<commit_message>
Fix issue with PHP's max integer limit
</commit_message>
<xml_diff>
--- a/tests/fixtures/data/test.xlsx
+++ b/tests/fixtures/data/test.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="244">
   <si>
     <t>bit</t>
   </si>
@@ -275,28 +275,22 @@
     <t>xml_nullable_unique</t>
   </si>
   <si>
-    <t>9223372036854775806</t>
-  </si>
-  <si>
-    <t>9223372036854775807</t>
-  </si>
-  <si>
-    <t>Nv</t>
-  </si>
-  <si>
-    <t>pN</t>
-  </si>
-  <si>
-    <t>JpYoCauprlwBtFzbNvwUYFLPeYMZIgitDbZDDbbKmbdikUtePItKGuPBLmfeRTXORWfQVwtyyIxOALBUvgsldNzLpmHZltuidGQTlfztLqHyHYqjWsjBNDGktzcaywjEdSxRNXZdoMnYRlrgsHfyaANGmZRCzyHdfEXgJvQqvqRdyCIXolkEsXWZVnRTYinxTgiMvbWjyPkBdtxRuNLBeFUnFvEcdftrSjJJqasyuSRRYElcUXkngIimDc</t>
-  </si>
-  <si>
-    <t>iYHViwdNPmChXUQMOnolzPOfjBjWUZVgySYPooDIbX</t>
-  </si>
-  <si>
-    <t>OZyWkrTxUmUGHktGMeuMSywsimnVxPESOaIsODQxYvFnpLsMZbgGCgPVfXYWkgztClmAtnXGjbmFLtvFXpwcADihcyEXGPMGGBbpgrTsaAYZDGjRCfxtLqBSKybJKtEeNdTzbzYLfXaEHoFLzIwqKERKgcvyyjWRVnMOaSoTpamfojxXVXueVkcJNLoTzznCuxoCpDIuwAAhkvqEWqICuTrJdmglgPtkHFEuHavxSifpXiuXNuzoCQCDrXALgYPyfuOtmXEvaXLFdNxiBHIfAyHEKMSBsuwodHpouoSudeKmgLjuMMEiyjmOqSBQVgqZlgTJWJFGhPODWguYdgazEDouoSJxtgrAEKrVEnDvuRavzCZmKbBPhpUOPVfiagWyBFZgjdTfresynzLhySwXpnBwtBxHpokCVUCcSwkZGEVPUxldeQRqKsBlAuxRqYKOxGvRYzoMiZFbBIiEWZREOAyGsPFAGOeJKqxBttdVhgPgjAbMgeSLffrbQoCCVacPlcHARkUaEsZMGrYGFHTZchrWNAqfThcuupKwxHkpmrhtNbKZgOoackiYyRRclsmUTjpsLvUNcqPJvovffRrhEOSHHZTXgYLPgnmpCpBnHNnpoSMymeIXrMCtwPGmUhbEgDeXyEBSLgZseWzouQxyFvdweBQQADuaWKKamqybdHQdtTqqjXwhOuomMLdfNSfMDtwzttvQiZtDCTYNHUpFjfFChbdBaoELJEDDEzHUjYQFteZBrtSuBtTamUnMwgVaFawGWTnHNhfeQXKVjqFhvSsIbRPZmHGHkVfOQOxBnwQsIlYgQXEOaGLiAfKMkcSlqSqPQLkfrgjbAiGSLSNnpqFxrukOZlrygFKpLPbWZAdhDpFlnVupjVpyYbNSSDTzNdHXSKCDrBMgjvzrgHeiyYdlegxCcmyGPidftaFotzWJZtcCjBbPaApuEEQEBPuAcQrhevAEJveSjpppyrfdjtsBpStqbiBopLQczbemlfWBrgRvlnALyrOEECgshkqEKkHBPkszllOgtWDILhLbdymoucxokBgUdcifHOnuEAyEzejdTcSSMMKipgKSRYGrMOvYxLtHKZByfYOiUQAVPhsUGwfuERtmnDmnFQAmQedDVnhjTovjgmgFuwJDRAbyKrmXMkOACGOzYoGaGidEFdPSEdPJqwCzCEqhQNrYmtuOpcpugvsRpPbNZMfjlpjfYQAmuVeGBRDunLSvHymZOLHfICTHThkGYcMgFmBOmpYLPkSJqKsiMxKFtGKZijXhhiNFiIHobWiNAgWrKBpgtDMUCmHUGUNpjZeNIECCdbcobTMInEhShonApkitNwCCMeCTTUuVTWWJXxvDyiZuVQkNSfSNemagRygIoGAVkUWKXlZVLhRfNUcJWMdLQyeaORryxzAoMIUDMySmSYHRYDGzimuOGGAiIqTJTQqeLhdbPssoXiHCovVTkXWrgiQYdecopmYHALbkxHaeKgPjZilsLUfdOgrGpfYWhAzRvHfumzpynAcuWzXJUfqolnxsGBpSmXAwvZNiFSfNVLVNIRsneDBogPESxfUHvcUadpgjFlIAETXPzpWGAHvvdVqsitRJajdaYyiicCIYELsctLLoiBKUnMQuIhaacxiOAHeDDXhdgwYLgKqhBuPgZLlnFhRnDcqnzjIJUvUDGmQtkWXhQdKXgIlmXbNOKiENLGQFskhgDoPcXGjgoBwJSKzfCJllVPUNLTPUUcvleSXDBQFSTjWIhKQxUSQKQSqbUcdzVZXDPsYwaZodCkffEuyLsiQzYlFqMEfRHrxYggwiQjIIPkEMGMjWQAPvLalnbpMdyHkqFWyvUvPIPJMZvjCAjizuCcfaBDyVmUuQuIdIhrMEzaxHLNcQTnhjWkuqGVDvtHIboUZvRymPSumeQDiuiVvdnsjFQRLOrGuEeCSpZtvUpITCEcUtAyOfeVSEOejQNpQjwwThdKglVdHvDNmKBUTbSTBbNRECxHprlXMCTnnPDqiALtROieiINnbwjblWBLuyNVJiVIYTSTdXJYqkMQXBuyoZJYGIFciqUbfhknQpRylgIxckoZFBLqIcxxsnCbgDVUmPcqDtxZkaGNdNBXYVeJrPrFjobcudJdYbOGnctowtyxZypeXlNTyikNCoUlLphcTdllhkKPzsheTlFqdgbmDAJZOiABbfiVCDqWvGalwMiWMRWqxDbclNmJIuaKyMKhchAmBGWGNKKTWcMKyPiWXjaDERKQTkcozKPXiFLLHnTiKvEvKtSdDfnchqyItHxgPRGZrxjkJeDJPzcAeizfFfGobAiIrKdpuxbdBtnZJfaMexaXAlcnMyEFseGqVoFhKgoRIkgdfSJDNFiqZhrQcsJTaJrKkPCkwfbbTTidnizGZLvbvyLSlndTeVTtnGJrjMnCmbMLumaxVvkgKrRnMhgFrbAJQVXQsuBUthcDBjisIwSTytBdbmEgoxPCyhQbaYeAbzJJpRXsOPhTxBhvBHwcBNiyIFQjsAZYNIkLQWuVkdCGzbIItjoWVkyvmJpImVaAImFoHFEOZkvsDfKwgtSeGnQEajWdenjcRVnoalRkTkYbQgKzalXmsxpNAJfIuBGVtqaXbIDzPOhKGtGPcMBxUXapNZnRjDSUPshyGCtHtTvkxpAAddDvhThfLOCApsmlftMYHuReFFyGFYYHFtczJqrYqdbXIdIWvykGRULnQRysfyKyQIYGXgswBgmVRsAGHxzQbFQHHKDqUBgBcrZlYcVQGRYWJbpBKdoYrvRzXWjMreZcbvgSeCSFZFogaaXcgdIENOIGNgOerFCnSMqTammrYUeeaWofnfHBPLwmFsOLiMOPQRMeAhKZCyWNrzoXeQrxvcMrWaqRWcdjKTEkDWVBdmouBNnzHCvrstQSpmdYCawbRckCtrVRLysXTDmAhuSPwLOCPVdUbXLveOQwWhrhQgKqXOVUzOTbYKWtFDwBGkEmYFWrNjCyeWhOUDvZTEdzyasxlkNLSKdDJgKujndQjKtBflhCVgcDXstmiCbrEiwJdGLjUfILxtwlMkkXoPvjIzISSnLkPJIYlbJZOiQWnsQBCPLIKYNzZFbCrIsNXoAkcqAtfAJbnOxeVMWLmyghGPcirxfWQnecthJLJPVTaZhlXPuSiDuCsQwbgPzLlxbwmFLHIoUaLRSGVLDlYfILcaIxcQefGdeAobijSVMDnwOBCUrknyGjYYSjuVNyPvJlDQumWRewcjzMeKkfJWWukjBylIiChmnDBKppXETGSEnPWIUBLhhaITrSrTgnKhdUrdMiebObrOCxEzyOXmtcfczHJtREkqpXPmeLHtjYkfppPwrnQldADHcrylHmDoKEMqYeJqrWkeGPKxnSADZBlxmuuDAnmdwBEyYZqXytjZSOeEGiwneiUkElMUXJGjNHEycrpebmaZDoAMBwvsMaZhFQSWVbGBIAcbdctmnRTJujTtWKXotWiaGoJlePTPxalxWvGMPuLBjyUbzjAmvgIuQPsrIzEIWgHdyqgnidfhJnXENUNlEapkvxTuZcqhHxCNWpWOWlGoepbReUvTHiFuAosakaquDNVnLRaIawxQhdZuRSuStScaonnOkGZxaknqwCOoRvbNLxufRsPBZSpeGnkffCaPxyciyKhaCPrKsceopljwCHmuOPVExeNzYGdisoIrciRsYGnCSdaiKxzlLQmwhEGbvsZPGvPXPElEoVsKTaIOuWYBRAUetczkDEQRYwuWqMSzZphxxHdvMiOxFNpYDlWRNPNGLKKUWJukMIeQIHbjcPEjfkvqyhaKkBLRtGmINgIiZuxVORvwPiaBngiqpiZWUXKeYxVFCFKsCEkGtxqBeMsjotvqFzNUfMMnuuTUsRdZTYEcQJSibMitkqjMZIrQRjPmOjlyhXzobjKJczkruBjBbpgLQoVyqWEStXGqMbqSNNMEuOyHPfKeqRXOQlUKMiAiOUVvDklrRhosdfLawOTFuGJYcsPAYTnCuftplcKyVTgmKQyZobJCbpxUpmqVQsqKtJklRmtAsDADTGyKFVxAEZkmQlBOyMdUizNSsPIHDKrIxvZHUJBkoIJOYRmhIRaYYWcecFqcetHqQbsDCoWULLeOaQWKYYhnTQqbnLmjFnkDuMSXXuwbKBEDeNgykRwVBeEgVOPfhuLGanAQrKHWlnbjnMOoQaszDVFbgRJNXvPRWKhVadLlKtMKvRotgsPsIkWmSYrLouabBMnvtUOKMtUmVtGTsgqhMQPWdKzrhTosgEutDNJksUwZkkJRHuUiJeMYRChMLHnccCZBBGgieoczfAcUshNYMnGrUtRDUlpaoCrJHJFdXPZLjKBlwvDyyaBkioqLkdFYPJtXtVkznOpLOfPtNjKkNOGwojEIzATSCWfgIiJvglCBqlWaqjVAbcozsqaPuqxtDjYsARbOpCiaJfnvIOvKtltQSffcHsomfpXwQXpebdpBOmXkejbBVMQjovPPmykJIfpAHyUMsGpVQMTaaCWEvKvvvlFKDHHiynHtUOObqaJlMAEmtHcboSDhxKbzVlzldZcDnRDDJuLhGdpRFfAHliyendlbBrVRPERmhYZbxwrxUpdPiJSRLSfdoAqfOzwyhAJmzGKvUculWmirntkAjMJvhaFrJQiNEwnngikhoEneUtpCILbgqEAeKlyjNaeUKEEJGhFjGvDjLzQTFLpqqBSuvHHaVkCRHZAEeUofFjCWbrJgYrIcjiUGqxgNmsqRrBmfQfYUYsKaNkICLngpMIJEXjCEnDheOyGQfNkqZVFRtLCGbXnqunZMgXSVIEHKWJeJqfyurDBIPDmoTzhrYHuoOtzXHxTaIJFaweIGcskuzSsGUZlMXpDExvJIVUWcvFEgarZnboamNuXQtXCQjaFFynpvzbpEANMTSGtkNzxfdDNEXruIhPgcGARHidCYpIoWvDDrNqUefnEKRaZBXFJExVWZmKyyHzffEtLhUBenrcXKKnWwUXbApdPkWpUyPWHXNsIimzelskliArIcNyAuZJYYFNoDTbKxIOxtjMaQoFwcncXDbNYnSALIYeWaSIINNOmefbPpqYnlCIXLGQPvXYBWaCVMsWaaNzTgrMMFxqSXhuqmQCPsJAucGzUaCTnLvwZWvxeBKiZrEMDrirwpzePPNCJyIvhemzwTnfxehaleooGqHoslkGrfAVppHCwZKmLFdNLjYEBdukLWkBqPgVauvHXvRnQnNpEtzJltVVZbfBXcQgziIhOfZabslVpTfKSFafQRPKFRMyRJbfKFxLNdOeiNKsBriHtUTgbwwSnWiLAbmszpgRqQuTqlqvphEhXeTElYOQtKDiPJZYskOCiVPXCHnvzjZnKmftbjbnRoySArJxpdnoayvYZDwuCrDHtKfEuasVmFKjbrRQmZhQanueKuJyjFmEHgfikJtLGOXmSpEBZoaZSruVrZFnAVGCiJoVyIoXxIKtggPehcsOjLBOcfKocKiRcivCYuVRxsakOxzwRqPaAXyrgSpQGmAXSctCEgvwlkXMCtcJiBkvAiWboTEcjrWhVLBdJozNmyMKJttTcusrywpZFxaBelYgrToVJgIWQyuTRpcUEGLFajyFxFvJJbgnFKbzpbHRUuUlJpNsBZPosWBkHwCnLrNVuAVHTmRWJFjIhyRGeccgkOPDpfmGgfZwAiDsXEPUAinaPMzCsVANHWJJIVILYiRCLnDtMcritfxqXHiLHFnAhhEyyvyTwQImwdoiBCLsFaZESTcJjddHpbMyrajGYlzjpmgxnTvFfYiouPzSaFyNVKXOPARRthjVftTbPlTmEKRRyrOnkhLbZDMJAOUsVVkqrmWRQRXYLBpniOfWaqeDLgLmVoHuDPSCcHzTQxtsogHaZzsxjVaXXQtpfDHzGouvIxPnBixcAokLOgImiErpvbnAvuvhihiyuFhjXiuivhNuMqQVHOiGCoehkNgVIuqJCJaeivdZZbRLYrUQOekJNbrrzAaUIFVISqquVFzZAiZAoKHYOIFuVAtFitAvjNmqnUabIKAEUaXxQpzfhWNVTnWDHVPQJeQozGXdwEWvznGZgkkxHBIDWSYNKKEfsbCQlrpvtwsqjdebHCBAPtwQLDSwfzlGjoCNcMvkPORBZOtoBGfeQweyHxlvKswjiFVbpNPmrZXvkSEwPxwYZrzTZrPNSQEDwEjMboUUUrhLEFNwLrwDWLwPrjGsOLBKUDTfFvKRglGGDtYTZiWzNqVauWGcdSlOFzZRFiacemRxTJGdJbnPvMIAWAjOUWLAmYbwzXFTozpLLbJqcMIhyfPxUwlqMXufIdsnnHLmzCeGgdhLruAwwSFTPtVaGtvxRgOHLbxykZNiQXxShCQAeckeTvZBTyirpWocAfEMCCpJhDhmdPkKepJkhsMWNyCXWeblEZBCLjLAwKHvlKokCJOGlMouUIvJMCbZkzXDwEaZYMvZxnfUpavWYKvUhYOhHdhcaPHEsPfagCVstQWGWENXcnGINuvqQydxdFvehcXYGLVvxMdmMTXXRtFeJLuIJZaZlDciUMdpIBKHCbRaDmDEBkUkrUVLNHIMJcnbxIxRxIPfeGHTcWUGnLxjvpifSoZmlMmkjlNLGmFtIehgZTwNirKgFxdEhpSnMhYQIuBDODmZfQUUwfVdRjSbTYplKqHpNOuflvydiftBSOaElFGAtaINUlqBwoZbEYWAZMTaiJtFDMbMJvfMdNfJMfVwzUSisdbeoGKTPpwJAhypKmMMEuSWMZHRXkjUooHRKvxnNynNcwOpBdsbCKqoJjxysEdFSJrKtuwBgFGZgseEqmhDadWaflvldvpzBmhiZzwBBpRqRtRykrsdXbhzOjlhvPcUWartFfaGhJOofEduYFLXyzemQhQwRshLQxTFRBMjNHWbPOOBRYRCpTmTAgVxOiwuqUjYsHASCZJOuLVFvhxGIbZmwcVRzaFgDfmXtNFUGvlqoqAvIxHynsKqrSzeBPLfLHCFXhgNNDxECjpUXcgxbSjsATuArgZyHUDhtDfbbTrTowaltaAalHSKMHgYUEkxlVziUIMCPEJUHATUQbsevkvHXEJpREUgaziskQqSYYRwVEpbTFIlzYXldwngGMaMVkqXBqvZEqJskJQzWZzJteJLAnijcCjkhwxexoYIUtSBIXNLlZMgSKLKBVRAibyXuoVzQBThxBLfejjIjFEbjFatyzYnPLChyOMSEUUOqYQXwUQuaSydXoVIPiIVrRWrXiOWEMxtUGaBAzPfsGyTzrOKKHNflUrwbPLycmmAsKpyOuGkgirDypXnAVBdxGCCzIQjTvuGFDybhiuguftIdWPUwlTmJfNEntHQoEEDSCbbaXveQCGOxzpmTiqqToZzSvXFddvDFvREmiSHgyajuGJhtQTHhBajseIfBYwaSQTWKZnbEOsVJTaBghYkSfmBumyhaTNeaIkRLOwKAViynSmmFxYdAKeDmQuyyFDFbSAhraqzZSCSITfNHVgpETwipgMNsLtjzpxqPAhPeovRZiOkvqAoEfLraiVAdVYMOnrkQdtHQLTjlSalGfZfESUshwsNjaudZXSDiPYFIdhKzlCneckmcoCSFlHRjkqORrVqMoxTFwnzmLadFaPPxuOxbgxcKOgXvZpTiLYUeJFYGltFQIvLkYlUawwMJwZIaAQCrLBflCaWduCvnAapEvvjewflvtiKBMtrTZzMQlmZCXhhsfTAOxMRIobrtBOgYvCUpRmphfmJDgjEQmmmejnYEEUhlbKSuchGRNUHSOtVgQQxcDjgcaYICadaJNhjYBcSakqHojkgteyDbshgcJviHcnfvyfSBuYxdKPOqUNUGZPujLltDzqtTOhzuQZavJORQJdfwSnYAbuyZlFipUkTaziIcfRRWEamvUfsVBtigwOLeLwVwbofHjmAnZVmjGMNDgAQIOeIOLaGaqiEfAlsiWPgIAFqYTokaPnLKMzjWPMpbCHiMmWUXCqCTJgbKGalwKsJCSCfaWoysHXkmjsHWqGSexQMhCYGVzBsfdkQypeLgfPSGaigyhTdoMFdJtrnnGpOngFwbkPTLLDlKqfkYJMUJAVdLNCfqCNFkooOoKlAendynPmjUuyKShbiXhzZpdEKWuBCSoeOrkEkKGXcqDHIfwdkxSIfIJGEWQUUavNhvEoeICgiRhRCKIfevqbShrEckSflNMiJGmsURzHDlRifpFXaVQJnBkPdBwWONiZUwgipkfblOlhTLLlOnYebyfMwIjEAcxIANmthZLHWsjjCmLgBOhYpQoWCUtkzriSHcvPNuOWgWMPowExQFdlSxcxRAdnovpmpqttxFhYWXGpYioWokVrOHYlfBVTsAAsxDYyVeRSsMpBwdEIfOjpJjvpqVLHWAsAHdyvURsOCpeEWuAEHzQGfFjJZJKqqYcjYfoYRxfXORDrricJOupdbgFkiizZROPRQlHNFDymMUjuPwvEOCRUzVMvLDZAjcPuANkpORcycYBCDxLnhboseusoUqIxekpmZmKKZAesRHqeXXjopjIFPHFoUaHIbazGMzPlmHkexEUQQCKkNkhUKnziTUbXcmmrUMfaxstKzfrtLyyBRsTtOIMvXUHUsTolIjDcyFLaYtQIquKVQkCKVnlGHtAwuMuGasbBgychFEOwrOjZdqqIbPghmTXrYhVpCFAdtDgohfZKHoWbvhEcSzSXxwXpJnBFrEyDwOinPZMrBPtBDpIGDkdRFLLoWLxzxihRqQnagvxLASNvjPyzlLrxxjNMgyYAJHjiZvCKnZjJCcXJTXbkkEiCxrPTATATdARpTdDmCrJwXJZaJAZfanmkWsGPQxxAyzWnEwPCbMyYeuIjfzMxYpuXJRChcqjpWYTEiIkmotATNXPdOttgdaoZZEhEZfOnrjAyHVkBaQijgncqfRfpSyoQwMkFGdfXUYCEUksniLwAxweFcZNBUlefpkWAxOPzMPDeLVEOEBhnTZuYYUMEKYextxUjdVaZRmSeiEuSbjIMtIzItROmeegopEAaxrAtCVpXEAXWiZpFsgBpywvhaoawIyQCaGgrllgpEUajCeFbBtIFycCHbEPMRMdpVkYPzXnURNEAwGdqPsGlNTZztDYMeNawAOJNAUhngrsiOAGMAPqLLuxDRcihXeBWIxQtouYAjfbYOwsJtGYwGaYoTAScJKdiacVuoxjGXlcuzKUtwhMbPfMjSiPFtexvKzANWSSPSypsuXUpyWZQXlInlbVXbkryNuQOXPEvpdDbUsBiprMcstEIGpvBEoQekZkPnEblVZDeLnoqVomedzTzzgTTUrdEqKOfTToJLUYANnSfOJChJxnQTPaBYIuJgeFQcQBaJPmVrGHseyHHpGferdKRaUNfaxpGuDpjZFtXrEMxcJoZGRTqTweCjXCkiVwCLXlUNXunyCbgGXrsTCEXkBpsKFtWIUwzkANoIEcpQaYWtCobDPNVmtXRyMDHoxwibdFLsNrmemWgDRTXoNOASBBKnVKyOqHZebSDxXvIsjqnqXNAlRMfdmdSVIRKuLZdszekfCLeaIdSslPPhtAnqGMdkEYUIahKLAOLJZdmGJNYOLtrUSEIiYTzLiliyuRtqeoTmuYWQImrEXoNcDSYwxdDdPrtcmcrGtrcLyePxqafYXmETnzLZqNjsOndIoVlvBhRjzxsQYNfCUGZFHQKCgAJrsrbnGDuiZDIvuHEpERfOAqwLKsAGLHteKChMpmvEYdBFZpwzZhPgQiuzsjjOJqzUuWCSEptTLuhUBXxufetkqTamznIRNCAMFdHfklbSVgsJILzoaBSgVwyDIQBSKGxPOSQJLdikGCfJtQayhVrmdLsWMLdDRSEsNVSfRRGgfTFvzCEyNQTqLUMdMlXkqvJecByZEUlMIULLTVLwMIbeUiyQUXburPxmKnUlsVauQWxLQkIxufJakOCGdWkscETWjqdBlXIivtVAdgdNTjmgVaBCdUQtndpwKPcAhAEwSevavgDukaPEufBHUIQWWALLyKtCxLdFdIyKtypiAbvfenbVbYPtTHVZAkBPOvQzayRjMulQkSUHMUMEbEUwSmLtnlPMPTXSpoKujnZkQAaQtxaZjGkJoKZNWHTUEfSQkqgQHUGBPngnxsOWahQobxtRnhCTsmbDtSTCcAmXHHGvMHBrRAMKypEpZIqGIcdQacmDIJsRQmnfxLlZWraVEcbSTRsQtvGJPFGAOYnfgBaaWpFulFLSLXlKXyFOYXluwYInBnNRVVMqGDeUCLCzepFfrtXiPyWjPRqmHpaLggMWEmGwyTGghxnmKYKkanlBJKszKKJHsmzVDOGQwFVzwOYhYyxsVzuaEYbtfqMACvebZonsknbFsaCoYJTBYBvroYTcXbSXfMkuksgSAxdBCydNSOXXGmWERRqJwcWSYKnPTVAaTqvqohtFZGUXhXaHSiMWaiDOoIgUWAhpEOYNDmlRwjNExjJyeIPRlHUHKLmtlMgpAlxpvalHrTemxxQmvzBjiBUGZdtHfEhMkMpOXsTcjynpAJcyPcuBskvasENQvmgmxIUpGaeHCyJGdTMprQEMnVMEiIaQOnHjjDFIdYxRiTbHTySqyEkRyXEIGSgxFIJtIXIlALPxfLPvGyELjmALywpbBHQSCkYxgnRZugybDPFykAzgtZUWlRAQpjLABZRVegqlbuIJybqGAoniANyuioysJFpKcvmiEmemLWlUhaInDYnSXgOrpXKrweYfxJLePBEpyXZZZnlbuOHNBMfmwIZJXTnCTHgIVFJKqbwWvDfaSXjRGvwzeoNnevzwaPJmLUJfVqtJEesxkRPLmNxuroRSygZnwkcyarAJqkjLIDLfrTUpBVWDPUyWLqGSqepwaQJPwwwDIciSnYANNNwBCNDbsxuRwGdQPgzrajOnyphKqnoodlIGsPrkXdrmGyRwSRoRepKCHNOwPdbKVWLgITOGkiwyFYNpmpWdhJGgABSapPjdtnhVAPWiMnJhpcoITLyZVhKPNqzRzuZtpnAeuTJAmEWtrhLuiLZByDEOiarIoKuycgKTGOTYJJTXEMhGnvfnXgkZZQruJibfhIktEokYgvxPwRoOrKCpkAqzOfDeIjbSTnGrLjGKhrHMQQiEWLTPuInJuSqyUUBOiVBsIjLGucBqTNlaLxUCTgiSfKDVKYvjsOKcBSCCNkpeVDcBbEYcmblIzLfOiTlQYcLqcfGGVjQmxCfWJPCjPgsXmHWOQNAugDjTYqbsnnpAZthbrAyjzstAvkFZNipXjofUWfGYFgeqELqxSkzwAuFusvThaGzcOGeyEYfinNpAvTGdhivUczFIoIOYJMDMaQqCRRZjTqyEpBQgPjmUqXPthZyWtnTFbrzWXwzgyrHRyfpOOfqSWzanNyKqiFtyXNqEYlPHaacGXAptSNRLANRduswFmOOYsyqVmZVzfEPPrmGQkKsYuzxixuFgTsqSfFpwQKLLgASkEyDFHYDSXgAktSTzWdMLcKrifiTBsfuDkhbLPlshnopmmOPjJexzwmskHIcOvhlSHIWhMgUyBBgpvNPzijqlVoccWKZlQXcRVYluiOJLXWgxEaQSaoLlHIOvNWhEJSnFcGQXTPGZiSRacfamPmTGMsauQepWpQIqOZMhGaUbEGjiSZffADkYwWJOwIvFPrdrJSsFnnblgNvVwIpkTSnSnMDgrVhgxSXwuEmCFDGOtVQCrfjadwTfcKQImvErUiEkILHBwzzmyOrcFzUCwtQyfCwRqeIlzdsNufWdlPjwJPvrmUjBeimqweRPAInFEmQJZwLZGHEbtmDeOiPUVTZyJSCrWyLYbkOcZNboXDeLaVIRpdGcYsMCiYsnQZfesPzkDaXQBphPmMqQpdduiufTqMxQtQLPfXqrMyRRmqdHisdfbqoHiqFILoEamtrhHYtkURTrcoeMaZiqEMrKKsKobwZntaWeBZRquIyLjjhscqmpvbberjWHKuqglNrZLakxmtrSwhilrjatroPcxVSgFscJwKHJAaChHXnjCsSmEyjJzYlikgTfZeqQtZUCLXZOZLlpAeyjkcmKLeQxTdDqKoePBIyilueuQqpXwxaqlzOSadKhZTUtLiAKNASERhLQQUcvKDkYxHKvZeijVoJcBqxrqHEAIJVKesOCJRClxpmCrdXryKpCTcOxNIfiWEBWvNxmxLQlpsfCrboQnMZUiqeewEaAXHiPbHGWsjRoSORexgBLMcHIlxLoYdInsnIoMBOenZqowmehTauHrevxcbBsjvFQNmQOnyvbCedrlZAZUHgBrbTkxYWTVlINqZvLMUYHujJAgdTMVHkpLmwyOLWNpKLobwqnVIfTxJmoqppFiCgyBxlOOTegycvlRHcsaxmPSkSyTQyLDJNYSCXjGOLBXWEJsIeheUqPvGYEPxUxsqHSrfVoiwVjpJOurYvlfIQUFYwbaWePHrFLyQPXbIYcudyBsJSpjHukUSjDEawYnItzqhOwJgFfDhazblFUARVvwDCiPDexXMSTqGWSlYbkXzcJIMhfUotQWvXAYFdSuDFgdqzmoqVwhGYUSMldNCMYbXMIvjiDLKgjdAkZpgAMZImrYucYxpZupvOSyDpQFOUvwOsbeclUuznKHERzYrzaXXivpnDMyqeBwaGsUfutkvoAWDEVIXbAcRyaVFGKPdtmZjSQjjKcQHVvXYdIdPwDAurEyEnDlaQWtqPFsZIMTQWGNyRmJROzyQiAjzrphWKwBgzVxOgXjaynBASacAzawOSUPTlhhVbfxvhioIailZpobXonkUhyCwQEGKkEBcEibTygQiWRwDMbijysxJnVxmiZSjCuhCTSVRpSVCVNdLqrCMEqMoCBkycyTAKSugvupJMpMmzxFSQYjWMgblwwaebWrqhOOLnftMggHnGOzWgcNGYZupFXncAkzBhwtiXlpZihfEdEUJGJBSxjnEqPGuYmtqHmPDReJtCuTdLfZQVjxkHmSacWUJCBDpitrCWlbJJTQvMpUGocRPZYNZhKwwvaYBQMsnAmYurKkClUbElIbQsqIBuLOJLKPWuqfxpQRjEBNrznuZalvOzqQxbFGXNKuYMgTjOactmahyjVpbtvZDTMNsSbETvRnZNYHleByalllkTirCOhBvlvjZITneXRZAAxAqMsNwETLMovLmeeQpfpXIUMSEtOnstlLUDalwLdJgUnngHiHRxdzPvqduBfeBYgLcRbxlxiHuIvgvTuoRdriPawxJVPrDasRqmPpOQkjUaLjVQiUzKlBRNUmNXWXNNCTEUsGiByhYZslIbDbybNdYaUVUQRIQDJUlQPdDUfpqhWIhhVNoXezYXysiQTYKIRyDjHqgtRfVtPvmyasioWbjhFMaMShWyAVwVZWNUrmVobyNZRYcoliBpxxChztswGUzAAVyllFwlkMdBIFApwgpmgymvPPmCeXvLDCyeqIFWcAasaCQssMXubQWDosivTZuWoFmgUvRXsOjhAiiIyCozsVhnNvRgvzMYnGTKjKkvcjpQenRvxDedLUejjZyyeRUHNsMDjvQYdmtxPUjSQJZkXoDogeAxMGOsxeSoEULEFxlZUwAXrGqPttcRMhQymzkGxBoDXWnQjPAdfVwteTAAoeTNJQgWjErLkcUHgmozjDXEVPFptoXQnWErNaxUQWQaeAbRIzkTYfLVZyqAnqCtTCZhEdcjxirOhyLILXjNqDbbNvqLfNhgyqPRbhenHATMtrUPmYillsytPHtCMYbFtgOHCgoLRmUsIyJXXeSBdzZbeDyWiykwAUPhOeRBnBIkjkuZCpBNMqoNTDFICRPrHfkkzkxqlnMWOTGSOQGQYilXTFzSFZfaOVVtgfUPYJDOYIehiwxVjjimlyYFcHZVKQarkkpHwcdFGRfDVLdTPDxGgcTdDDjEiVZELBuBOCjnqJdwDMTvtbTpvDhyoQklakjiTBwAfftdLSXjTwbzoTnbJvzrbvGZZJUmYqPYsCMZCUkUcnskqoOQHGlOFfHfSYXUpQnhTodgDeJbDOAAbEydqaAsPeWxUWYSvXkpNvlDcqwKwKPKOrAcSjnrMQPdIKotPXNOeVolUDjfkpgkjRiOkwSqSKwzoqLaAsKCZToivVOmqRFVPjKJQwIcwvhNHVaAkuQAMwZDgpBJwVqITPauwGPZnDnIcZrbmTqKvHbVcakWXrHbMsEvVbbLzWsQObzHWOXwDDvLdlukxTdKvaZmsPmaCYTazIEhSHfThXOwJbmvKgxOmQpQUjrdnkncNRrmGuVJxpGXtGgZgSeIUrnyGGxfRiofpVhcOatuuZhmzNPbnBVpnmCNIefSxIZJnTuKkXPIwutTYQOsIxkgXdGUBTasAzguKtfQRgxbEGVCGYoLlVcGjmBPynBfFHbYQRPkCMaYraWKxIOxnngGcPmjitPeGQxXOojPoNpwdZkDTbOZPsblmfHNCLYQIJYgsqNQjmyiDjveXuCngeNzvWCtyLurrPQfBjkjujZbiNEaXEEhUzTBMeITzdiWOcgIbsrEiPRKRLLPXtxwHiPDyGQNAYAEPTGoqwEzIONCTAykLECToCEhGTOOWLbxIctZqckkAXGmgOQHBwRmaZMYrgEWkCZsrtjRbBospjJiqxMkCVwmWkOWyDQkFTyokoJNRZqcOVJfAceamdBKtaIhXNErDfcmeyPgZosOdoCDZEKgQZyVoMYclcgURouGKJRFByGdNncaEvojKDYwtHuoaiAlaDQqBXbffFlcBVLVZUmoRhkcMXGPwaxtDSiQWDWFwhECjnyxNNBjGOqZuBKYyBMEpzJCrztnIRQVkABAlPBwTdgLYIUERMsEHSuWHDzFsYpOiHZZzQGEhKTpKSiqoOYzHrdYeahtxpusFqGRqFIrmhMQysIHczRWcLTaOqzHcKGGbwMxrYoNjoysYjPlMgQHVxumQjTvWHQxheGmScAuVrBvaTDuaxvpjPaVArHpnixIbCCjbycijHHStxWeHWYjXzivvlHSHKbfbUPVXoUAcYTOIfKpDsDucGgeCyVuKYPqcbsNqwIRpovKDxEVoIAYkJuldElJDApFsDphJqFdDeOtJxXXJobzMeXmHyknwxsKsZodRCNpTaceCNdhrbTXEnWPcVAfaWxaOAWaAhdOLMbfkFbCfCkDsFleHnwGpeeTfcZMSDhQssKHPaBBoyibwrbViryLHDkRKUCnBGEuDSnxJXAwZiOkEinNTIrKHzkLfLShQXYDyrMtdfuCkEIifXLMnZCFtxelGujJLiWrKyoOTLDwKrInMYAXMTyXznOSjHwWrliDKvhrJtWwyArMnPWCXiNssYycWpJXtEdVAQQhKyTJfjYyLYKMCJRFYqhXcHmkaZbhWpIcNAOVshLsAlBIkZJmBEIEFsTUKfsXKZAlHwirmwBSDBeNdzFGCJJaRDUALZhGXviFcepnvBvcZUalWNMPJJLGRkkUWiVLReuEcFtYhPLPqWGtIMUcFSTLDtJInfFVLcbzQlMOBoJNfSVBKjCoepapWXUSAHKzXpcKTYXxCWBfVgpDhSGadZhmwgDbsKtNdyUXLoKbZNwIuNZqTcwsfXcWNNzlYKJDMJGejNEsoLbiCzkGleuiDgMbuzfqQEewfQtxNmFnVusKIehNkMcCgjUQVgpjzTvkPkLZzJekubPWDrUyizAwzKdlokVhnrryAeEpSZWzPCZYibNGflCewrxvqbQXZEgRrUIVBmPEMkyhBYfvaTzkXHcnLlaNxwoCljHFslVxQnrslbUSTSvExCCtArCRLhlcZuTCvWsnsfJbDSsIjyIepUbEQiFXJBtmeGZtToeOMTMQBwvHPwsdOXKOgBHKPnGzSLIzEkQlBmwJOVvfTtMmtNCwLPLSlpLqlZTzrVIiZgblaprayVvTZdBuXzeJklnOHmNERQMWNxuWwhuEJEfEfAhFaLRlwPRKAHunKRXrDEGXxtNnVVNjYliisHWCLEzkcZENrAiBrISJmAkKMNMyrJUGPryaKoBDkIRLtDBerwywAzJAnKfQpSauzZErmSQOWpAwDqSmZsPbkxKdxBOdfpNgFlkkumixUoaoUherATEhsywjQnAfSEWZNmMeuDisRKVhlYlgTlmHEGgvHeLUAkAEXsSpkiRkYnnTkWLQPTdLvdKEFLbyMBeXqKbQazomUkuStFcMARtcNBgqhOeJznwsZCiUjGHemRDjmqGsjJjtOZIAioOrXNKBytxOSzWesWhThQOGKsNooKtIghwJeWPAEremduPykMUGhnzhEwceVdvpkDtweYOEzoPrjaLqEROJaSFITUEMSwZdfSFvSvlShnWtbgcsIkbfHHVMkKImZdwytXbDCnFdwvrBWKANIkXiuVPSzLHSxnYZUxyCBJEHNhKHknmbXMVuKNKBwYUIweWYThpXgejwntvffrwcgHgJKaQzBlqktEyNnIBQHcFjAGSHAxgDREVWnNzmTVbAMQGTJjIwHZkJigbMFDXvldreYgiwATYKApyTZbtCRwMyQNslztfHLIFJDgHkvmHECqioTJZUyqFBlTksNrGfuBwgjeCeNvCcYOCxouusVVUAbUAciYWOruVrdEMRhMnmTNXKTkcSegQWocyRfZyGwpPYQJEuQqhgeUvVlEKpcJodVrFPXtvZyTxZsIPzgVhrPyHMbOYgrCSFeycmvpgdYdHomgYmphmcSfkZFwifpbvXUzFnNgRDqulKhiXfpZmzUoWuIVJEGlGUgXBQOZhlLwenzStqEgOnHfopYJMQfaDALVxzPiwIYqeVqUCaeVxGQJtmZctsbxGpmQYdZlFgYVhXBZPcySQGVMnpOBKtzKWqEEAoLQTXaCpOSgqxjuIDCksyiQYRHrJHXZJUncIbxwTTwEPKgNhCutNMWRUpqkWqDZnZomGsExUTMNoSEXmWWqYEwYQzPQALOZKkEqygmyYQOhVazHsVTdkZLgHJEIwkByubqEwaUqSBpMnFrQCRkLeKSuPojiHQAOEuLXjcoPktCfRtfQWbdsVMblJNsYLHoMOYJHDHRpIsHmyKlMOBhMlYelzfjLGrLFnnrTTTnBSapjOEUYGrAVPnXmRaXYkuSNmVDiAMPDzGNzTDUicIFuBRdGzoIWpvrYYHMRpImcPfsqlNRrUVKuXLjVwCkUQhykKcHemvgnAEhKAlHndmQTwLWrRexfDkBIhJgKGzqARkrLRHpDwuRcpkawWoAVltDjUFweZaZoCVtIEqiUmWVGdNhhMIbRfAYQfQNciSuxrFxcFdpRHwqCgwqtAjvIRuWCkqejuidXfOQlzXOVYWNgzVgDejXGZGWXzQEUlLYJWihcsgglWBATRwgvPbKbVOfvLdLtrWXWGLLTHKaFSBvHuWHhagMCWoGJsWeqkJioUiizOxmGzryjhQRUydhJuCSoEcNaWSCDgfzfJuxQDLwzMTaJQLjTbRqbcSBbNOKJBlSKlFVPkHfyecxyJDSGBlmQxSjqkZEpgDNgzGQBBtkYoyqhMFKxkqFWJsObUoTAAOrkoLIbBcxePTdUmtTaNYkCMyaDdfKDXtsvgaQZGULAQoHVqYDVvTrCNrYCYqulTxcOHlaZZPxoObzhrfXnvjRBhgdODvoMPWLOBquCcluuZQkuNSDQCohEprJrgRRTwrMrpitmIItmzArcmOyJESodHXbEscFUmJdOCdCPnbplUphINvbWFBGXgLNUEegfYpBPpalfARyrkQIqbdwGDbDfAQUVNLyimjFXOEsdtByqarcdQfGtBYgCZasUfyMvaYOPWFkBAJMxugWYNmHaYSuhqYUDDdSUuQWXLBgHtwyonxWPHAzqFoiFMOIdIjDmarOjYeZZQUCpwckIxytWKUWkSTrvKoFCuzHfzckNvezcPKDUOgnaKvkcGJPKsQSKvGKUiHRrCaqxSLSOKIcgSvSwBTVhfeCSQnWINUGwEIUUeFEHVfPlJpdoHUqgcUKsjFfuhHXdthcWKORMQSTsnJtpowvRHFDFFCJKbzADuaPqJQZhhtUqsiHVuxeujqhTzCIeRtkXioMPWmhsNgSYiGDuqqoYJqUZdwWlcjnvorawylxEweswnHSWuAZUVJuhRCIkcmvBNdxuJJZQOJrHIbJHGSEpIPZXxJOdroXnnLAPxhKMKjYsUclLvzLrQmgSkCAOupiVJBNAcIPvNKcJHqfSrFjGRwjGAqSqPrjmFMYCyCejgADpTmJZwmRofsKoNMoPSbGrPGEHRbXAPlCgrCqYMaPptUFXnphyRbJruzSWAVqJtQGLEtjkYUsBEfFYZWtOMirfFHpqLnJOIfAIaCSFncsfmFEzjRhjwRxCwezyyBUDEQUujaJRoQSxyKNMafjoSSngdBCwWlMOACcqCSdYjyysmxybIDHhxcwYXfgoIjblgYjQFkBnoREdsXupAOGCioTsRXsVJDhVwKGNrjdnmjZEEZJqKiEOFsBfrisIaJIRlXtihGkCHbTJeXIQJMmOecbBKSfJCAWdQOyXgGglIksKnOMkOBiJYqtGhYOYdIrNQZaMGGrZVcEcjAWyXWMyAtCUwvfKfnZjCvAUhILDkkbpOAytVVcdBjPYbrHAYryPtiuUmSOzCOLQwtYGBAZIxnZKlTzhJVfPkAlqTevbwqPwvOytOIluWpqmSYvksSPJldQxUKbkobTmINadeujmixFRRzfoWimijqTNzYTqMcUuQgnFUbHgdSFndyClBujGZdZDgYMextSHgpYCjYFzMabuTdWAKNKRbpEeqolqNXTKaIZbfpSUhgUeiONjQLuDrwPiinBupepoxAadVrZDGiemXJeSzuKuzagyilCSwmqjgTfehXPXnuKcGrDgPpdtjklowYNrJveFGQPrkiJhxjcdpsVWcRdjwvJxEnAFkSTLBGwHGCFGizPXKnweEWuwOBBgESgMCwiWubkFcVgseCrYxjERhPiWFKefaRvkfTuEmeLGsoUGuAXfDdNADiILsqxPYYHEGZFgaAhXbUniOFfKAxgxXpFEzTfwKZuUhQOdxzYbOBQptAkbHqhrYwHabjTaDNLoclQtMEShaErvOKMZbfsquQpznUurVLnielTxzPwTkZQJsdLdfMZQvdUmfxbfATyzkfwJCxKXNFCGfKpbQPDoiFQffdvuGZqGJVSBbwpsnRYIYQUeHmEBGTVwxeXfywXhdxFeWnFRJDUpznNUFahVGcfbTWbpPGcybbBkuPTSeYVgFxgQbHcCqHGyCgXvutRLHcguEStAbyqzfGHVrVkgYGpdijJcWGTnnkqeeCLCCNvqCezgnPImWBBFkPJOMgpWayhPGKZeMxJQfIRjmMXHngtWHbhseXcpIEaNfxzBRTSwdqFSOXzeyrgrvbMZyUQlxUhVqdeBZXJsskPIeRGyPRoQalfTYlvRjDKqzoiAfxeutSrTOGRlcFSyofGhgHoxtmiguEJjfZVnxcWyROSQPlwDCONincFWcafXfZcYrKRyFJKjrLPrQxMFEhQgmPGriJribetEDfTESpPOZkZZzuEwnTGXARuwSdEkOTvRBtVfKQaTyNsDLzGjzKBuiWFrgIwBMNLGRlTamFfwmdWFoyoQrEOEXrOjBsJEKJUFcGKMwUUXDXlWfyGfXkzNhRkVAUxLYmcFFmWAUWDYctOXDDaKxMKWBBQhZEBgnDtvWddchFvkGEBzDTRRVKnoaQoCZSvzaWxsWALlUzEAAOKqsbzlSysKAYXxJexIsDquJdOcBlDgVhQBwXXEUMXryXMePjwOualzVcTTvfKIProNmbFKgDCEXweonfCQqYQpSyACIaLKMWkrmHVVvCRTyuWYxdTpmCpbvcwJPumlfPuAKdtbegRkdmIJogpCzeZzrtVTrbSYKDLBgozDmdCToEvpORXSgcljBXBdbFTIiEBpRjAPLxtOdQjuXIjdFLTWJDLeyWqqXiTlvisecRqMtTFJHyTHSpBrAWJvoglUoRsoDUYkdpFnlvuaHlNJuauJmaTtwnIBLRbghoHWExGoDmIGABoGVhuKucIaAVTSHYqAHtgmqQsKVOmjMxJBMHfATDmARmmhBBQEshjEEHeoQBMZUUkaFnHXNqWaAgDYHHtjXnilCWpDwsfCfKTHwzVlYUGwlUrEWESMlJCcstXhrBRdCRNqFSLtMdWUZrfBRUTJhJqQNSmPSXWZeSgCggJWzxdZonvrFIsWdMwDjnfvqGNhzavFXbcEpvShWlKPsskMBaCRhFefuaFsjhPPXAHuiZSmTYDHBBkqvORdHmulIpgqXwDBFcnhOxLUNNooIZysFukmuEKARXOPVhXmtIWCxVvFpHjgeZEqzfduVIdAYGCBrXXyQYrDsKbXFLZhJxvZCJrxYEeSRdxvULEtEdtKEnBemECbAsDjNXiIZltDBaKOvMtcfkVToMOrVerQpCGzrtqINdwdogmBtjrpQoYPYFjePtpNvnwHQOFGhnkOGweJbLUFCzdpVnrxgbvncwdSYYRajuWIBebPGiLpaaKUOzFhpCyBgUhUrMSiqLTgvshCXoGSZgDESVBfSTdCipLPZENPfxKgPhNfZYcKmxemzHFmbaPXgDeJeAJzttbXqDxNigQgLNqbgTMFXDUgbQRAmcvbnENqTUmZKELmXMrPqZTgZXstvLQwCXLTBaDiBoSeHoQnGRlJFeymOxJxTQiAWAVsoRABkvtkcdqyARQsHBMhwzUErfiQGgDrcKgszbrJtAQRvYKZdlkuSsNdVtBCMnZnZGnUBmgxVFAqxsWJNyxMxBTQYsdZOIxRPLNOKwoUzEzePyOdbslXJSaoKoWgkdaIeBkIcspsmgPFsZsIoeRFsdklhwAjVQrPgnapTwlGdZJpuqYlUyCIGFPgMApXMAJLZYrxwuFzVNmxKTTuHHWjsvKZbrcczEPzMFkgjfNTUEjdVhDZrjTLOCRBNeEmfCskPEeeMEHBuAmTHmUDWAuzOyVlzedBSDQHvStLCDBpPzFMagFeOUIZRHYtrzuSslAqyZXCynlflFgIAmYGBzTkHXbILPMGJqSwmpSJiflsYSkeqhpnsxnKNZHQwWYHNTVsgHaTGdQixkaUPJWlPfOwvrYhvvoPeucTYKYrjwNBUFqMlomwcSHLqYpimSgqrNMuwqUEVbUlBefVfuiwNfwBLNKSBgaSaWqgOawXMYlkJqUlqHBfUkqtgnyRgsLPEflJQgrIUMINXdFyupydcWFzjltoerwITWnNNAVeRZxWNNPMPgxoZwcDriWgsJskSIhCHyoVdgGhqVMtScDlNZYpCXlBhihZnAqRNfaSDhMMWUEBXBVohcNWCGEfUYkgtajbOLxNHMArVqldfbqywNmrUbyHtbVmVYNfSaVkHSSzktKkKapliHeHYQlXPBxbFXuRHMKVENlIsUfSwlLVPEldiceqeDFtfZYqAREzDVtcfeHXiKSPLBUCZPDsIwSQUuCXCJCZjWkcIMftvFyqtZPSJzCYzVUuATvKDTnnPIcJXnAeizqgDslrzCbhbqpDxuRLxIKNQZnWhbpkKgmOXjYWxYebosNSZTpySmwOAwYrWSrOsKRJjpBArfdsEyobcBNqvToSkoBJPqhFSMIEXAGmbiAoCnpNIVgURbyXkIFcYzeDviTAJEgxUOfhhYljVKPPiVCqmkbNutpfGwdbliKbGdzYYmPGOKPRoTyHRNYmCKzrTiTYcweGaecPaUwpbJaunPMNSgqgOPPHORBCrrSXVDhyJUvPCFEiiNeQKlREaPhtOgRHrfNKtxSKLMIUZJsjXgkaXJxeqEhzFPzFlNRQKgPOrvhSEvckubyJGWSZVgzrGFZCOOzzQEHkWFJhLVoiRUveLWaUqZLzNHQJjspztTFAnHFUnykcANYjNfNKvOWqwVooFFKqswKaGAgqZmMSDtseAqYaXOXfvSjwLsmEssbtzNGJUvwMTWMUTfmAAEMqrDVIUVCuKZrAagceAmqRTqHFyNoGJnoRaDVokYbraQYtUuwokbmSKzVHgFSYnuewABlOWhrVIJVsJlLeOdlzKlGDhDLYTHxGOdhLcRBHQjhhmuHYGvYxirBxvafufXfLDOzVvdoDGZHZHukrrYcUfevhJBIYqSSQQtjPWmCdNqoXdHbCAWjiHabGFXnBhtwHHOmPzFyyqKXeuLbmZiwiWpiCIFwtQOotrQJXUTTAvbXqqIqfrQACYJdWRHsSudgiNCzNXRDHBPVlPReBWoPGWOdAZWebcvinRFMvahxrJFAovyEXWDeJGqJFyLzQCiqymxUyqLtvDOrysxKlouspvyijVpMuQfNmEPjpMjUWnIWnQZgGfgzAHHpFOmERTbtsHeTwKWphGfXeHZGSqStFdjEkKTeBIJRiPVjKITvQHJshxunQiCRlgehkqXscRlYoaaUnCBeQcIquMKpLpPjuAUcCtGpNRADSuYKKhuQaIAVIaWZnCmHGxEYNptLlfstqZJbMVcAcKtBrZvKpXGRqUTOtDOsQCNXkIRZawbSwBVUBxbGsvOnzxypLQnADDaZJHcxAUlDSSsDcEeJQqvRyapxepPcAjpMqKrfPiJVCxEgAmFcrKLnaWXGhDMbzcAUFFWVEetTetlQZcDIrLjAWhRqHlCaYrjAhtyasavIBzhmJehLDwuniMmyUYvZbMpQqGKBGIMkLKIOCofATunYWzdRtOZFHxkqvGXwaTTskFUYZhzEmwMtCCwRAXxWknkARinTJwzMnEVelMMsOTJNiLdjtauTxcqvrKBufwRtDGbREGdAyIyDArItHCBLvLWTREtLunfZzJKsMUmITlILtygLbeajgZNAeRJvqUrkthOkPuGMBwJfYRIvauEiVrRuZkoHfVcubSBWMqAutSwQOhZjWzPvvVcMRWXipZJWFWrafdoZhBDrljIJaETLrzgzGpCtxYQqAkRqFNDGjNCIkgmqTUvfbikUagWwNdrDrpAWCTsEnmyueDZboMgXAcpIpoxszfpFTUSYnjrZeoezicMSJlzYSDdethvsUDbZeeupGjLwGzhovNgmyBYaflhbADvfhgmOfwefgWrWpSaSfzNeRhSWxkrzFcaqroKbarwvbxPvukcEOLyoSNjlygDoCUHNcINbvrdomUzFwtrNkUXBsjrelEInzNJLNrAhimbcWDgfPoSbPikiwVwdrdCldhCbVUeWiHWssvuAOFqBKuvhGTLKwAeWrdRdEIpKkHQRqOwGczXeYlMyehbPYCdZnSuYczLFRQNCkVAFkCMvzEzrqaZZYBiyDtZsffwOzillFTibVMqbNLSRdhOhYCREAxFkYSAzlYGOaanGmzVmYpFrqKYlSlcVGDnKFshGuCDhcdfSzGiWwAQOrCiCxbOqCjwgdiTSkQmCspyNqWlJELlReIroArrlQhcdaNdACmoZsGAGUeeVpXgOAmmkshMoizEjQydvzxzeYhWzBBxwkBKtoAIvYFqbVTFKqejRWwxwdwtrBeUxzxYPMtJSydCrfEpsucbFtxrXHgHkHsxrJLXcIYTIePSxyFBSBVacTkNpgXhrOLkuwoDgznOdtCXkLOItNOJOZHMByiIfWsNEWRPUnedqnVIqcXgCiLmqJjTGEPWCerMTOLhWZOwNkWqoGkWdpWttfEbWqlSuhnVlJzQQAcoKXOEcnQpgIdRzLWVUUSjpfoGoPOsEynqZbKKnmXxAlqyJTKWjiwvsPXSYCEADCyrXaZgZUNQHGylQbADImfLGCjwofkHwoKolMSPFGplCEVquiIurRCstsMdivuOMgcUXbPUcaPsIJSvVlNBTQeKnJNsfMdIgQorNnrFyUDaCcqLLxtVISDhwzcUTHmGGmwnSUssLoIVUPPzNbfQkGewwMVunUWEOeDmjHCutMQvWLsJnTAJlHJeVSRHRnVAvjCkHYThMTOAuzRBJkqIOFWpFVRjtAOsyKAPQJVMFRRYaigWapuGzQzXEoDCNKmiWsGFSsJkzCTTWiGTTCfWXgWMOtkWfNeQQyVUxcNUnSfswHMBGODSWbevXhccLnXIERhJfOWtImHHFCeUvyhKxQFsprKuulYCRiOjBTLtCubIcuquSTdotLlSsBlhLeQYoFfBtVmvGaQzfSHjhNkzVBusFggTGzalQTSRYyojOmvKsDAOuBFVOaTMdDFoCxWaslMBnhSnhVpGsvpVrLuFUvCxVACKZvQrUVmimlOLdswyKbAxnFsDBbcUfolPgGXOkaQpozWzJYwOVsxqvnNqjZBVySdPKjfreSVPchkFmCYxexXGEzebeiwUlagkbAUdnzCWJKspMgSzbJjjpJYTmYdqYygcQDzuaTEfHojDqIoQWxsMtnmEpinXZhArExGdNQzyjKdQrwmDzojosJNFyVjxEoenWwpGldVjDYjvhKimCjHqUdvPTKHROjvApEFyvlkkLKnNBhIPQdvpjcGMWjqFdrwjFoIUmRiBuBHDCcskcfxgitvSlDCrRSwlUQrqhUkYaTGkDSdXIESjjweysAnDzJzStNMlqvGRZGzNRqfVmBwFlutCXZxOlNOkUbUWcWUbseHGqEYgsRqDJUrXlwUPiSZQuvNqovvCPLTISyUZvYsGjXrVZSBxbGctoYZUFoKWOOJwZPverbFuBrwnlhuReUPqlxQMEbHZZXOfVsmuPurmwEiezlkhtRZBGhCGAZBQlGYLJrDFkOrdsqhzNyJceAynyWNNaBmnCPtNVHRKxEapzECpvsZAqTYIAzfFzCmSXefUSFyMEvxrKBhJmBlbuvnNXxGJWNsJiAruLXBLACRrltJqZvOGNcPVxtQzRcYvANgJkinjUVHXkxFNVdRTGBtcSBxRvfRudHYfhBQUHERLoybOggFFFvgMiGtrKYwOvLNdhwiFTuVBhbVNqQnYApHdFwTsnFtQVFdjVrPeHlzuzxzaNKiXXTyHEmuDJpCgRkilHESXJFDFAJtNARKGFjrHladHMFkYzDsIZKFlvwcrxUiaRbWaiCQXfxYdWlYtqhBuTPUWqgqywcZOQkofpIsNjSZTOnRFuZQzxZcnzXngUXmeqWuZjUCRcMTnBlNBRKzoOrIpPKsBphSkJTGZQhDYiXgqpcwxrGJJBqwvJQgfNZyHraeUIGwRAhBDJOGRbNGyqUvBvTVnGxBoFLRhqiPwpoQdWoQBdpxFnKMjJQKvSCcASoUEcGZSnqfnQrpZvkPSEPAEKuBdbBobvSLxdkgBQKDggdlwzulRFRQmWfeisEFuPdWHYLjSDHNaYwCMwoIUxTiUjowVKAaVcnHuixapHrTKJmxSyfUcYeZlPXyLqGpxtcXIPPOSpJkCWHNscWcEfCYMILgPYvPCDtEHtODeFKrTdDlxzsmeuCSRFkCDKvtIpongmNadIHIKiehJwyLcuEykiyqVvyfvauemzzCterSpZiSERoxPUhUTLgpxEvPcLoknIbMlRgbxbEXlWrbRyyeACUxfUrDWqoylgHMBtgsUiAuAVgsgipKriTTSVpEefJJJJfFzMKkzERBSGIkyUXwztiyekiFelrbDUGqlVHzaaJHVBqHQbkcaleVOyAmsyRgXRkPvhdQUbaODGHTOISRHZXYUohgfmAwnPoaTpoObWeURtVGcQGRaPjxkaRmWArdgkckiaXgSlfKXzwLQsxSMxaOChJFCybdsqdByAWMBHqCyMcFAGSuLBdkCKvAMDzZSaZuZrlghgOatPNKqSguuOLDRtpQvkqsDWNOsHJRfKhKOcEwAqOGfMetAzgJvwdmMRnqchbmPyhaTexrQelTTwOWqUqOcvQXllDTULToDpBLREnaEVShsNNfTlKnINBBfvSAeUeKaQcIhFMXWOKXLlyreAVueEdfdLiaZTVwAGRxNBIhQaJMrsnWGiJJvBSPiAuJziCEibXWozAJNWtswDkNVNavWXhvBtBoTITZFjKMfJgPMuLtfJLVDUwCNtgQbLDRtlAPcVFGgIbPARneCPiVdRdtBjWbNHecDOcziCfqhIjqFAPgBovquydQejFnRvKBQIFkhbQaFPmgZfvFmYlOAmPMnjqQSPZMdZRpVqMVMLPfgftvxALFPNqWIsWwhloWJRJyehCXURhAQizNaypWYGbvFJJlWkUJNAflsWQGKiWDfRTuZPFzXgbbkhkOiDQjVJNYOyygHcySyCrmAvcDKjMQOmZDCjvfRWaNrWXqxPRvstKSuDCzfbMjzNngFYhsBjeowLlmgJieOfaYIhKRgfdGJcbQHAXmUXKykGHGpENAjlQKrgwGOWHvibpHRWlrghObtwsuHYVXGMsSmhADEespurqvwcXDjtKFBNyMRxHIALIrmXCIhfuIcMnSBqdjMeKNuqwzOGgTHjHNYmbHFdCAlblhaXUxmdWgowOSfPXRhUvEqEVsFYxJZwBSPnwNgFAjePHpSdWDRLPsOSntUjECAJcCaYqdyObvKSTKXwkQtUEqKIbLgEyMamnmLHiffwdpVRSuCbOUUUujYcEzVufqgwuMwdFWmHgKAgjkNHfMnEfRVcPyzBYuPSTaftYJSalwFLwhKuucFPBhAfryhCzfjutPwcyahtcYhNYYFfEjffsHmaHXIvvdqRDtYsykOwkjDxycOOuxTxVHUJUMwiBtMNzsarpivHXFnnMTNlKLIqpuferKinIRCQhdXjhcOyfFJoiSbXMbbLwueBNNJzqScMvlaUqKCKPOUdWuKJpZCFHHPbWDxGdiNZhfBjeVRUSagStyxbzIaplYuHjLMtyuRKFrnfksDSGoKHuQiCBUvmIYFgLYopFpvSJPNjDVZrUUirNNaJJYWPWBAlghGyHFjNjaikVLrXaKUgJcOoEDTyWkZoOQXwliFyCuXgqonSwkJwskHelUyiDOCmhfBZPyAbaGZsNilOVqrysUaVEavpNkeAjUulbbLSZTfGxeukbNOBPnEHeGwkMHlxDCgkxfhaFlHntkXfPXSLMthZuOpKLSrZQKuNlAXmdwlgJvWskNFyudyPxMKbASzoUpTAccWugnEPANDHcfbCMLvqzxBEjajplufQwoylwJyxDBxctqcQRSqvjBRFtMYmyFPjOrkaceUsvqBSnYynRqHccoSOqxeDLOIyVirbOBkdxrayIwbicxIVEREaBoaEZTESwZJjytkTAlhgkpdHvrUVMsdWeiTgvUQxZJzEKwFJkyQiSFQtAKfOSVsxKbstItSvgfDYMoXrXcSjJQDnRpdOmlZcbyqkHKzmeCLfEPbkXLjnNTQNgsDHIbDpJoCNutuLSviSdmiKsCIUIlKzTmsQxmqxXRzYmIzKDQQCeTEmYCKKYUzfmpreqtjaUGrDWPrHFNVBYFJjXcouPTHZyaBnlWYadlBYlRrOcgbYbusJrQRdRToLmkEDsFpeUbkuSJvDmBTPnwihcAzzfVgViniXWbtzvnzGALXcrtKurJLAmEgpDEGwKIuxqwBfmNINejUIZZrjLJEpRQOZFgwdksmeCUHJrwrWyJTxiPLWkZBzHgvLzQajNWyddRlhwdioUocQcakCYVGRObsMPoncdRWmpzoTvvlcirQXXSYVyAeRPxjypzVyOHIfYqmnVXiZBrYnuTspkOJwwpjwUezeTRjZGDAKOsYgXDNcQTPJHXEtCOGLbUDeuAedOLBTzVICMxynJgWGoqDuRByXEWBImqktTltoYlgrrBYiEqEeRyPkbctEEErIigsGqsgBoqLTEpmqpzkBJGVKuensMEBbTUaqkJQxrNVHlKyvDgMSheoPjdQQcvyjcprWkDdUsJxKNWhYYEjSOAZtWOeZTvvFJOHTkbIHjXfmFPCxUHxIHfzzaULHSrjIVxyGfFYjVOouzpAWjuMktytwJPDyRwiFSEScFTMEvhbqfzbLUltvBMoegFoZSUmzNutgTNWGoOYeiiZHOOJPEhPtJIXOIMIzmaigAvlwiOPVwROjDnUzjsQKiOCTDeqyNnKwQKyWwDryWbrqRYtOELTAGdqTOpPmdtlOqsJXoCyfllyJaKdkegOVfpaXOFTPVxfbtZKILzjCWHRTQJBNnVEfAfUEZYlBDiQpykqeroMEtCgSQFIixEgfaEdXqFIVnZKjywNCPyEmeVRNFBsBRHfKDaKGiSCcIlmVIwQkObaQovNcPvPuJjNiXbNXzpojoKTBjtJdlTKRkXPCiRduoBluBdwhVoUIBkmgVWwUxSQZsKnhvkCBIgIvxfXxhYzqdZFMPbCNgIQsUfJFBCpsNeIJBNinyZgunslIhgJxoxZemtHldFalPbBClpGdFDZPqEbrcqKUVQmFIOAyteFnyPHwtPYsvbDyAnpaqZKQqQkNhHLODLSYOzbgvpIIQLeUAyDauGjMuMIUFVgLNnigbbuSRzCBkHfOjBBvSAHTZIJmekHKSuMehGVNebwrzrQWpKQcABDVZaMbBZUfigYWZCQorKEWNMIoJJqqbjzNZnUXoESlJKowTozMBKCECGvOgCsRlwJXmRtxSahoOEuRtLaFHMZjJDhsClSbhhyrEowydCmXedEJAizreBaYfQtWTwvhkNJhNUMXFJpkOVttzsunZwWkPdfODNhbTlYTBThbjVeiWppQVKwUgJGxzDfDyRUMVsNILWjEuelVknGFCiSeWdIfyrghdFFVfYPokMRFCRJyIjObdeBQuAXWKDVPndHEVouqhIQDOYIHBaCUijwSdYOdORDsCIencTtLFRRpQETkmWCyKPjEEeYybgrGnQpoZxXTaQipKmZMwhEMhBEElrgtRCgSuEQVgBeNYHMHEDXvszYHGDxAUhGaqgBCwXzBEnKtWjsWxZMhGZvYtSRzJcNdwhItWTfhdSxeRlQtVQrlydKZmbuJAwjgZoWDmUGduoydHTeYDsGoddmnHhZCNcmZyiaJmUrxHSbAroKRTnRIMytBRtMWfqmVMUUadMqmaflKVlfpfBcjEiCKKkYENZAEPKRaJxLuRkFaYMsfLCcwACPAIpzuqRsNtzMdVbFhQSJQAUmMBIGvZDCmcmovaWHhCicUJTYjNRxJdAgUbavQobwWkWdTtRLqBrdNDpMTTFdVvKaYgTearsxzGBihoDdjpsCmpDgmWJyCbxGyWKGpEDzpgMDDFRPwyezJpnXeqZKbjLwHxPoumOdgTqxJnvEzlHedJhGBKfGwpAXAziiGbVlmtFaeujMmSSYkLFioMOgspMzzotZyYWkQKYNsGRCNAvQZaaDUuYeLOwDgMBxCNWaZfAwQJUbEqvcVqltpGMBzyykhreitnuUNhiuwIPMTQYQupArKQnZDmKNbLNMYOcQDDTvVyniJbpOBiWdLBDZxhMVFrxkOImemlWiwDjOjfHNIDBPfUoYMyIfKZWzlwUZntmaNMzHKzMLlfKezuHwXngjVbVlcSwErNCMWApyLcnASzxUzXkbbXlOpDxiWRXJJhApsyNaTqBDCxDjhecLvIyMQxKvxlgqjxRjfjlJzoDvVgugplvMDjSLYgVdnBiKSovqeSHnNmtHhWGFnhhZtFcgCbDIfspcGsSLrmjYVCXDPfQTcGoTYmxamZggnLxtWiTeIeEtxsvnyMotMzGESswzloZGpVacMxHwsRQesCiilrstBJPrTkgXgRMdkevJOfHsTaCZMeUletEhYtmXmduMLaVUIXmRoGdPZmWPciHkqUgFjJhQlUAJGhJiAszDTNwsmOhovTGkJzbwwinaFHdRCXNrOhFmkUsHoxxXRbvQHafUGPMHCwkFywhuLNztkZUEWAKHiTUrbclWdktRBZBuwebAwHaCwQzGfNNPhnnWaTACLJrcFtNQhCxmFYkXKCvqQFTzkofeZVOHUUNhILCcznEWrcwMBYKTNjAFxhIbvaSMueaNwELVqbtHzWGiWoNQzpIMmRWypSgIAbWycjIIBQbiMOUFxrYgVSHgWQcAnaCEAIfRWolOStUBaQVaHduUIUDNrOJhYNmZbQNfBNAZXCkQTbOpeQGOwugThUSfYWNSBuQXBzvDtAcLPCIcTlqoGkSCsykFFhomUiGkzCauOqzceWeAonOEkmocvBAajtfMAwuZPEttYEyDXmvSwzDSpRKjHjiCNlKOfPgVLeuFFJJMldstMwKnoQutszxQHgCJzVRMQZTpDTxMOfQjhGhWZMFFVTQVRETEIdyWlVIOTaEWGdKvzLuXazjoclfoeCpDGvkeOhQpajoxcHZZDTZVWVTszuhRopLjQQHNtxtnKxxQXmodvUoQlKiwuQGSSpMkhjupRGyTKgLWViwvRtTsZFXdxHPJDEgDFHFJWNswwkSynzIRhqAbPBRgQWpspvbGrJxwSbAxLiMVCPaTBYRAsPjItAPDCYQeGFGCliFupiChuIZjASZkZeVGscigLTCAVxxpKncjlRnjPvVLwFNsFLxzeeqsmbWhoTYfeettJxNNylzUXtALOqnywXnwHQSjcxccWnEeGjetXOYusNOCYPzpdxjDufSXOyUSJdqhbYJWwLSORHTsRtUVCoOzwPmpvzRTjFIZYjvrlXQOhjHjrmRuKkMbWONzMhZmLZeqoJIPoCMkpkTysMCNHNmGTkkdcnKCOyLcJeWmjMDZXWEfNHhxhkkHoFfMsfzOSauznLpftMdMeUwjLSQZmMKEoiLkadLCytFGMSyUQPezxUWolaIHnCEkYxXsGPXGrMdkMbPAetdJBvwjfGIaRKwYZbZWthKAlVfAyZeOKchpIiDbGfMcEldkoczYHltTduqXpOefzmYHFdrFjCbuaGdXkrEdnLNwiEWvjcdcJglbOaFsNvnMZNJKoZBxBWQtcDMlqofifJCNxtmbypAwgLFhImlJTnANIFbifoIQpJYNqmCwNOXfLMuDhgSxdCtMpaRtkgNOkZGENUMdRkowUwcNGtyOkAZwnNPYkwxWgMXUipOQYlelocFYqjRHeOzextYRgMKWlqiNLKPXuQUSmkLyHSXfsTmbubsdeATetrDupMLCMHCeEyIRgnOLpXFCooeiDYsrXtcWrDSxHnmhvRQxcnKKdBxDPYYUeAoeLTBefGibBsStjUfyakRqkYQnIGrXgWKDWJMXMfZmDGijlSmCWbczTbeGHLZNwYfvRTQJspgivzzzUAmBjIXRgnqCGoKugZGXCutvQhxmxbCeSvSoXmuJtPpRaQXVYOnTMuTCNoExZhnjaZukjprgkouAfroPaVWJYeTNorPBJemjOqhhdlsfsPvqMIoBiYcIrahECtOOZNulGERbqUXLtUYWXhHHnQpauIRacldMgNNBEFsjSvvalETdLBbpvTpSImbagrQaDCWYncmRUVVTHvFfvDDPVATiRViQiDRghhwchooHdnZpbRbhXXNsAfeAYZJqIATjCAqQtPyjExVjdsbRXzQXIdpBlEjIuxtVbEerAgfurrsCKdvMaZWKKQGffXexsARfiyKyVemVRWxleaolIOvotjTUCtFuoCfAXyjJOJYBvxtSFnFGLeMKzNolzhSpAXILmXXJsQTLlWfpQhsjwsfuImjJmJPKjfgWDDYdRJUgrGnCgsuoGqJvdPIujmMfYhXEvqWHulPZiEtznGHwQgUqPmxtiznVkXsAyUtjPsLntHNeeHDRLEcvGQQSLAfoXabLcDeHfbZQqoKCOXWQNpxOgbFuMrPovgHzGcvePythKBztsCFwmFJBtmyPRClnuRigClxfDwisAaaMoyRWHFXkNXHkobOWBDMplcxlTxsDzwxYnRUvyIFKClsWvrgNhhtkhkUqMAniFZcQaWsvJWnAqoOagwODdubDXaJGrxLpZYdBPTCTZwqymsNqBsymkpFxIUHGFYNMewvHUOTxBQZLpnkUhuTYCIRLidMEFSqMbnvsAXOjElkLUNFkxgjEQzeLYzEkklrJIoEdoMYuDmuyUcskDTjsHjCNpTQHGtZFqGoGpdXPJXHDUjMlexNVzmPxoVhypoLxrPhVoAZRdHNeMbkuBupsLosYyMQtbuiisUaLMSUvdPqDUBOlWFjUhhrctPtgAvhKIFgdwYPiJYlByrrPOBJVBAmmmQTsSAMiTOrkQaaowqVCbFqUOZmFEMwbPLgzPtuzjiNqqaSEGngAHNGeWpUASuxsRxLKPAmaAUJVtmXJdcQaxSAsYwAqZGxXybvUmAjiohlZqrGLuGExshabbyDOZoGKczimqQNBRQcfXyBkxuGzjPeBMlOFcICjAjROLlbAUDqDruatyHrnNNLSFWHjjkvvqAUzWONBlSoznmUGpTMpwAOcUPwXEGNuxFCVxfeTEvzCUCUIiAQHURemChIdJYynFFrfryJItxbYHtpfUfhYsHPeGyntxRMZCntifeEVRjZxbjqjKVjMEhdESisTEVqoAfLYrwgIQijJzOmFbfZkfKuHGtTxmQmdzlrHOrvdJYXYoiSxdmxrPDxZnFCZyGcwEpOemGyLFWqGQYrJBpEqHzZoqDXXoMUhuCIVtxhdZETLIIQFVvznWWkEnrRWEmwehZUSOwAaDMazbzNFmlaVpyuhcBvyJxgMBgpLVCDjIwHldlBAobQRFoOwvIZBZRTSYGacnPwPWgonEhfmHGNbTRonhDQuEjYqJwmOWkLwIuFCPQuclnOXkFNeurJazhJrkQIuUVcdShYDbvIiJwCCvlvKHRwJRRivPzJYrOOIBrZTZrHIHiIOezyhFkKiwOmbnLfqdqzPLcvEExNTdrUTbBPipvpRUJAhdDknlQiDMruylKywbJPyinPgRAOqDKkZWZUwaHoukgqxQWOpCstVIkkGakOhnCRXULosJNcXaVAhIVOHYemyDsYnKbkyPxSXAlpWleFnYGcpwKiXFIXjSAGgimbWUzvIcCBnux</t>
-  </si>
-  <si>
-    <t>TVGzJGngoHBkBgSkigfIDWbLLDeyVKYJwBIFZoYuwKerkDNctQblbieMLNdflDfKsPKouxdiVIdFsIFWngYpiKfPMxsxCTLVGyIEzwfzyfCXSkdJNBZcZALdJAhwIbBIWGNMcBvjwHvCAifoUCWOFaHrhvJhpNQRFIHctVobsOpBQfeFdLNSzGeIfeTCTyZhAkKgNHcLVFImoIcWlvdBjJnEgrvQNrvICdafyKKrNNicjURaXnpeMgQvFCsiGrYPWOzUMfpDYMGunbjIgzAeSbukoiItYuBywGgpZvXmUnXmzpweUCHnAxjvpKYZJbopXaJITCOxbsZumiXmyBaDQmVBXcMqkhpaPtXCxbkkRZVAvsZZoNNzZwVqmITVVdqfwZxYWjaWnASjdaXXywPYHFWefWPwgJdMEIWIaszCFkDlonrFihaAAjHufPzIsrYJbWSuzMhDrEnAfZIagUJyXMJGTrANLRJyyhTYMwMNabYITHoTfOIxQtmsJBnTpOqfsZHFtTrfSUtoSAbEvANbLJPqvpbqxFXHTfPOUcKskZqyZhHrECoAhxuAMppsUdMikmjduWbxyVcKpHnXFWKeozdIOIocGQrDZYjYLKsoIlmsWVsWENtizYmSQSJoeLNOUswAmQzozLlOGOXkVBwcWcDNyvNKRvEJgfzZOiIFKAsYdlhBuASMDdwtuqtaVcBQVfMwkoXWVYHPUwQZCdgtHwKDbtlOytKshdsSAVpmlXBYFexbyCmVYTbkehzkDkPxfrzMqinNQmipqxwpKpBxbnzulzsWvVVhSlktJtBOiaKkSDeRCaYReBGChosMgGtCfrgnLKhfPqquRiFjxKRkTuMhkvuUfHAmFEryVMxQegDPbZdVOqtCABWJgAmBlhrCvwKbRlmbKcdTdiByguEqAUUMfoajvwcjMQOpmZvkJVVixsPrMSUgExxbfeNoXjnWbbptwlsTLjVtcEMhhGgLwHdswaKhUbouwPJqOzhtpBExQYHfiJkUAyICfxksometwudRzUbuNZMHBsxGyAwMwWVEwlEdsMKJNCWenkjdGMHYHtIFMhvQGjzzDZzmXKRAtkomStgcHBuBKTibjyCWUcaFvNroZefsvZHKOxudDmERjXEpMWglfJsjXugfpdfPkjEQhyQSwscvJzBZSsxHfQytKjCnJtANrBcWVHrJLbSysjWTaYODsmVwMxWQyrCxrsRmuRGDqbKQKAbhQhMTAGOPYFEimyCYSSYVTVmcVysUoyYNidWIzKAyKcfYYrmInidTrJGKRInZLUQJxwHxLTgcuuSYOqwoqCiELCnLHSkZaoyKDfxYpUuLsQhkPgMHgoJtZXxXYuMGXplqbdoIMgChnCuuednGfboytTQHgwkWYNEBZNKUgvkqACZLhgdmSNuPGmjYTQfwMHLDVKYrMUuqDzJLjDIUGKxONjLOJuhDVfhwEwAeoKRPhRZJDwMumewIAGWBQOXgKDqQxvJGRsGjqwQtvIjMBcEsxrNzGYTHcpYyYIqUlZEvPTOsjfILIuAHQHmTmDkyCTtzGMRAtTqaIpdYLCmavHdETqWUdKloSIVRKBEiNgCQCPlUoSkzAiTgztgJfaUvXvKrlzWAaWmXRNHZNgPZoUiiRieQAkdSxPlplneYnqTDUlGrrQUmhfUIAIVqyvPMoxPlygwZRqLdYKTXydAVDkXILTRrzBlsLPpZZxhzKkDufnLDttCkDcbnltaWxIPlNCIgdHrUPyTpdONTgOqBSgLzzhsvCqUVPYIAPEXkkEaIKRRlCwDGzCljDzIWUKzqOhWvSekSjhnDtujeaWGQEftBoIFWQTyyUUkFSSOVMDaGOBoubKkjmyTThyPWTdaqCeKcoggreeybhcyLBNcAHXGqQHKBfOjnTljYsEQzoQAWVZPJzQnTqGpeToKRkSVaLVwkEQFlKLoVOXYHfRcSjVGniJmiVZTtrZnMRRDqCQERVpgQmlpQnHYqVIOwdIZaVwBLxniLlmKRGSYFoZCsUZryWGyfXtUnhYZsyXplDojiAcNRJoUAWEbmHFEYSXGqmFwitTBbJwHNNwsCXBBVVDtxeGHsjUpWArrcasdpnJEcjVpZpnPseWETxaAbdkxayPMtfjLxeANofkpvLhBaoPLjmBFBIvwhqXUXWsyIReSxqnyfprMjwcIoluATuqiImAgBGabjbYRVWqYCfdWVcXFmFxLdBuftHItryIzHfYssSwUPTJronJlnzOXqGziUEablxcTGDSFcmKLRUcJGbARmgXhSolTIFUsgdMgaeqWavhgsXurDuhbeYtyZTSMlRRxFGaezNUMrahbIJoGXcjUlSwtcArqEniiNLchGTSyQOfNukuPBHWXLoVhPlnOaBciCaZaJVbTIrSEEkkBKEAdjMlyLHyvTwROsPQUkuRaOBayEnFzElHQCePCudrZRemtuGTSQiVBqIwowRjeRyrbgBkOeHiUvsiPtsNsaJbrVbKoDoJvlOCWXaCcnAFDvseKpfZVfgNBzjJzZBFQgqJzeRFkvFMbiArMRmmPFcmuXdhPTnJJWVZfpcQbndcdyDOHRrrobJXnouXzcfsVRmCEcKdeJlyTzHzTaXSVGpmXxLKhCivRLDDwkBrwhCamNujqupTqRilyeCQUEMfFGgAYluLKWjrxTnhROoBEIalPFLHXYNtdoeeMioLTOpZrrWYVYBgfZDKfoKvPATnUyloHbjZHFhtjpUjJPsWoZGTmcHSAhXyTNfvelzhVsyfCMBQjoYENeLquaIVsnzDFqDADqxAxmUqXJIYMZeGhorBYprFLwzXqDbNrxmQSzboZUkrKrVDxyMfNhiPCnBlPGCBACNeNLmxdsDuNjOxlgyDVCVSJVzCfetWDJgnWAQduULgLuHmeXjEOJcjBlvaHOKIAIxnwDHeIgegMXPsksWqWlvkSMRiDdAoOsHbDmCpQFfUGNXObYELYNAGCtpBCpzXUovTOmOxNnshhotUxTnNmTYpDRBPvfxWTkgQAOxzDComWipgMqjLLXaSRnKsSubDvxJXJKQNLgJldUMGHvfIFhSYEGjoSVspouZvnIcYsEVzaFhbiShVaXfIYCFFJLMvIqhsNlvIeNpBxzdrEUFFtgdfJWFTGUAVNMUfGlNJnayyLLfEIVZdYVcVfqzsugPzpcfeQkBVMXTSZDRddjrpSHaeVaAGKFrxKUseyZckmBJzJXKQarSXUGzdGqsSPYAbriuxXHzaIKeHXHVsnEqysaOQlNRXyboRMnXauFLgMtnsaMXxRQbtufKdOTKugXnLotAOHcFygBuQmyQfQyWydtmoabDQSYlydzCxwClISBTLogosLjtwLKaXuZCPvpRIumLkdEPiJpauqQOvynFZTnsipAkpZklGJyisSyGPHjlfnLKjCqbDBJfKJqNJNSAfEcTbZrCyyeyfjLRUeKGfUOlMvQLRWiZpFhjBszzlQMisrkKoKuLqjicylnlHVGJvIvYgbfqwchjcjhmrVZSusTTOtqMNsRfeBnkLPXmjDpybOsXptPotBhHtNLkkHuVuCIiRZAXtMcvjLDrZndElztzkDsUJzYKcHdaKOMIRUUfvbECacGYWwwMuaDLhcyxOJWcRrijJnszjjaUKoQyADZvOTbQUldwGwgTTUUrMjEnzrGxkUlLkyUzrnVGCtlLufITZLPSNbyqsvRelOkhZJvdRCYPlxOFVzdKbzQeHygOmEsWDJuhZOqLUSmHdJAtwJFBtTLWwLYIKUGRnbFdzUyCBQwMpGxciGnhxnMBPZBTwYehlWkniJLfbjaUoeWXKYvxmAWEGMJKicXIjuACYldzgCdWzRuNZkoQglzYZxqNEpKAIGgSmAMClLiqKmXtnJGvSIYUpkLObmGmogxHlXcCVZzlIYvcUscGLNtAFCJtbSzuLrUUFiKOsDvhSOnZhOrEMnglpsIVaDLnsMIsrEPqsjaXmcsYanHBYvLtcSsdaSRFfiTuWADOLlZZiVTAAUBRUFNloupnHcUPPWYzfZGRMxGxrXXWoWVDyrzVtKZBIqbEJWydTuMSfuBVUztVIYISbJDapgDnDwQCUNuuaqOMEaHARXVFESxVruoeCyXspsczeTsQCRzvBcxlKNrGVaMiKuXouLbleHTkrjAiKfWLzJmVQXYpntEGddyNHgyUhfMKDUPegBFQQJZwClcAlQUZzBiwPrYbFdqsETALDsMZvptmjVJUsaaMZFqdjPOThnyPWMlpdzWTfEjNtLTMOYnHfdzHAUrhnfJbLmdBEwJQNgqnKldyyOUQWPEEujgFoNrPEffhlAevyHkeWdWBjyjKohMiNfthxvXXATbCggIyGVMRbMaKzheeCmXMYMSWSWAEOCzwdAFkSeiiRyoZvApEJgmATgXFueLXdsxLcfTvKRxYgtxQPWqDcDDRwcFAnAXjpwDEwCaYUFBclItsMjxSAHLwUOlDBPouGyRIwqzayWCibyLKJnLYtzuqUPYLbeyFOXGnADjkObsgNNPQntTdbQCnVGziOrnVRmgFkxZoQILhDiMfitTBzqjhRbOrUFMJblIPkuRgOYlxFZmkPqJEbysMPQGUycUrBVnrToKaNZhhAyQOsKijDtAklOHhRHRyKsMlyaakYPxGcXVoxKGrooGJsAyuRZTcVcSkpqdhVcMzXQjfngRFfmazcNYeOLSaRGnAspjPyHHtPYvZiZbNMkdvxZZgplknmpYtTlDfIcvjJDZxdMimciMUqUKttCqQCRJukfyOlgvLFUENGBPOxSfGgUweYYYOEzAkHSxPPrMXWpnfgmbpdrRiEQgxPfyXdIcoBSurzfKSXSzuOrmQuHXEvyGVfYCXlAphsgcNwCzAvSsmdGDSIzBlQSoGhlPUhbBTMqJdXMcmQeFLqYRaxTSNIrFikMTkbTLjQeOSWxMVMfBPQNHDxQSNrtDIrYMyTMxTaLOGFrbIayFVHwUIXugJXFqoLQMPtsQnBRmoVyYZXsFMXeuVPCZCPPBTOwPCVrjIQvlmsYtuxblCsgUAbvYfuXhPEZonfQvCiGiRSlCYyjYQbLFgDmWTQkDfkorLhLdFoHvtQghXOxKmyJOmUobOcoGHLwtyyhwuGBVVbaUAzWnSRFpDlIcRmYOvhhArPHlJsNMNPDvIoPufXlWbCsaQxWyJfHTnutPPucOfvQDRnzYICtYPbjNWPwwJSTzWqzbhEZeyWNDxLKZXHHoFZIUJgKqDaiYnrKPaFPuIBASzxgNHggtPwOcIDEYkfNxoXLntQfeiqZAGhTssWFgDcrqVisdrEXjjEChHacbSyihOfXnWjYhaJiFTQkwefbQmlhPlIHWRISmorhVzVOYvmSeXYXchaLwyxgYuqsBOBebkiiKcwzuKGDPGlkSzfJhrlAYbHGbggTfRvGSRnMENGzyQoTJqiEIKBpTfWLvOluoYoxLeVEYUrJOCeqVLbondwNxaLeTjqfkAHBYRktXopHatSFueFaHdMdZNfunAynNAKfVhPnsqCNWhkFFIgDDYOcjysBSlhdechJwGNRNaFmlnvyWHNtkZJjryJqVEtcmXuYeBBYdXFHMNvVwGcvWBPQaddldOQsmTlCRsVnrGFlMOHZidzVVfULkoXTclkfjyWxnkoSqYWxMmymHRsWCBHJxVZWVhncMeAuYvTDlkAnOPgoPSlsloxoxolgKIilDgLMUuEpDObrsRgxCUnVuiSoKxgaEUvjwCPMpwwAcojuoSIiWCedJJDTpJfqBvDMHIMFxCQAgqLiUPiEBYEoAjqxxvzkCfkGFSdiwnJynCOehtZKEItfSZfeUYKDZIqMPaYfvZPRbuRHSSXPLsHrBCDlzCpCZYphuJvEkOSgCYsiPkeThIHwpaeVfkfjepqWstDezlWNMNfzitxFlYiJUNvecBZaOTzyBUrKNhBALzrOSkTBWVvWyUuKjcxFvTxoyfMQkwcnPaMhGqCUHuBVDGuzScxyaaqQiUMaqsrgFJjjwBHjSdinUQOdNruiubEQLKZHmyYOltTJtJRFiGlYZLbMYVAikZPvKrVCfqFgOEBhFkQJLvWEZCfwtNWOpJtzrKQsDWmuPwckZWTxZuxJGiqVfWdFNkWQOMXgkzKPFmmNkjSCbTwBybSRoSfwWeISKyjULfKWHsLTZXKEEMGUbiMrvbSUCxnLqOUZmPFXcsGXWOwcwRxQMxMYvxmzgYHeLhgCIRgJXVjUKdQbzTvIMzVhovIbCnljptYWgbQbXiVaCyaDagqDIzyWZXbpltLPDljYtNuONGMlOjlsJEhoxCCIwbGDWUaHFPvBnIGfcnUMYHkjynWqjgcFUMgYNewBNJbGRHSrTZgClislUWbQaIJYrANpkaqvOfKvEPFLPujCGiJGloqnlWWOdoqczBdYMYtAhIuqKLMlROtQQktdTLbtpIRSqypgJqNyEMonAaDflMVKBgAFOnUVSwxMqvdZJcUatKngJrZVNvsfFBQrFwJFkkrNjmaqQlXkHRbcEzbdVIrXpCJYRvmizkYDnJfbGkVLELxlYpJESQJmSZczAISlsctAJbvqlYPLobScBxMvjvcdOeROrOYVkRzHsKHlHEDqvmwBAzhIpclKRHkjxfYYhXAQaAnYnVyHtoVpIWvFPztDgLghFXqEYTJgvPYyMhAZvkWkRuHQwzeCkRrtNHvytmipFXGgUfalNnoqqQoyiUSgGLpzxJMSTXyzujMdTNOEKukPVfNcjToQDmdctwoteeXZCkmaldhKilFFWIbNGAMgzBTiBudYCQJGBcbRBogtWznggeLNDyuyFCbZgpuFRsVUVgSIsGDBjoUMeXLioPyjDsHufJaOazVBlhkochSmqmLiMxkqWIRtLPKwaKLTZzoFrfkxxkxlhbmFxlaeASSuBNKUJufQTOcRQbCanBcIKmwJPLGiNrRYjkCUllahxloDcrvkHsIdIOllLFDzxRFEzbbMnyPvljjXkqmDitbKzERSLmoIquOPitGesEcXiWWIrxILZPrJbDxsbSGWuCDrgobAKANdIHyrmTQrkRZLMoqejzPRgSZdYuwtZYebmCkniEzpABKDFFDrkMnzMaMHQZWtDngRpBjvyhjhcqpsBvKNqxQPmBhBaoWCpEQYgcThesffkmkTpszFBMBcixbSSrtBFADDMMPhPstDMqSSkgYracDymJgoUvxcoxJALfAjkjRnmdiyOecjUDStQHHloPuFnXdaPNXHNMXLpsXicaNoWUbiBXDvoOwbzjyOohcRiOxwUAksgSTosTkQYAaqXGQXRribszfHgTTyPWOGjHSYubbCudEfTVQaUWCZBYAwOMJPKVpLDDUCOtXrrUBLcOVYbMGUBUmEEtFsIvPqcJKiLFggqpKoqNKvOfwaZiwwITmjJBFNDuckPGyRxKhxDqiWTcVzvVFoWijIrmvwMFzKmqfgHWDLiilsXqWQMFhPFMDDwRvuVcJippfXHewKtJMrqYOTPTCeFmplbYlkeufITqWjNANFozlOlFdoQdLWaXnDgfPJwnfXcLBmZaDCbOEZQoVGklwYWOuxibhNBPAOYYSHNhlgzeAVMJsxuoCkXRNmcGPliePXxgxlYoMnXcVHYsiiMqqlXYedSyxGHaNUbXFebedQKuJTHRrqyKPppxpDfckyKgMvsbFTtKnxyVprPuPqwDXlwADVqisUdyibRZKiCAUuvKSZZGZgmEyTwYHnVufawYdVqMLKUxDUvkTIsYPoXDGwiNFQxVwqGRisYZbdUYCWCaSAsPqlrLEXqWpfqWgCRjIFbStKZkECPvhxBkwNaAbiYNgUcQYwppcvoCkHdiHuNUuydxKAQFlyzmcbCElQDfPvEvudcdmXtAlrFfmdPlGNuLCGfDwmPQleMtXcDxOJJDHDFfKKCsDDAmoActRgyqvTePwHzmPXSfgnTBmShJHgFwgQajdADQPhXPUEHmfxQUSpHdraDbKxKrEvYPRnUUMgDrbEpuqPGXSpAMwGcGKaaUhtKvMHQRtDVKkJCgIrbONUCMVDyncCgLdSZQqSPKrEsPOgRcDBjPjlyZhetVPefkEPSxFOfTheyaqptTYBGeqciojhSxMHkjyHEREfRbZAcIbWmefpschPfywhLDYcAPtshRNThJJRpxcInBxTGlxtnTHWkDVGOrNqaRwaxsUWoxlQrhmrWVzYazvTQnpeaPbloZyuwDpcZULxImTPOaSuunSBbFIwibftpeexbwQsYJqcoezcqLArrCrvszgHIwJebCSrgUzooIPtRWpazIEVPqkyPdTYscKmCeqHEKfiQNrFiqRIsFxsxAUGWwqMaAijIRQODiPOqAJNOMYIegZTBnqgcaOolvycCxrtjeFGWiJJAvcjPKCMrhhJAXDaUAbJovJTCCVqKztKIGpdkhRPYvxlrTeafbfQzhxxwBfclyIOFzMVNdTPgPXIXqldCxGUEJisInzlXxAOfcwQTQlXNyYpEQCKTMlbbBcMdBoghbamCkqzJgyWlORBBUFBNvptjoCWeaZFcAlxRhIsWSXBiwhvpncKfryEroUulOcGNyNCFaocuwyMiOoAXCCjmhqNBWnsEWNDkptxhTzJpicsvEzamyKsZVYZLgMzwbjjCGOgkivoRhwqAhsociFcyTcinKHxGPDBQfiSmJrXMTGdZiEoNrZcqMQenaHjybPJwCmZTgJLaAilHtAJhwqPPDVYIuDHezLUoPnNwYPivEdQyWcZVLtZJeXGtyDmNZKhIeumDHvFJcZZQIAMqtzxXbZlPTQAAnuNeGTzXbLydVZpvICsTLZywntKiHkmaDGXvYOKmhhcDzDiLKyFjlEtXtZdVbSTfVauebQoUdNEMEnMDbxIfoXMXFSWKUJuIFgDUrYmemvWeINwKTpZsiOzDrydPHdnjGdrZFTzVyRVDxzaHZMCQbLqgJbxdoLQxJyPkEgIfyhbTrlwzuoOoKLfMeiKtrvHcTjbERujjzowiRjDYWWBDwHoHGGZNjudbqZOkviOHUjFwJbtNwpPoyLYMVWnOUEqvkFKtUByTmPeYsKbOqDtdGlILChtttAhwQUEFTCAqErxqZDkJEIOvADmmjkVArcZZNLlUvKgjGzGCNEAeNznyfKblJpOqGKncYENPFxzQmlAlGGMqfvqlGxLEFKgmBBFTknNvlKwpLDyRsYhDIctGUgFoxPMDwCDDsgSaNnvfFmhQgerETMiEUAnhJWrjqXqJIPyHFhULWgwiVEmzmxWlmGqEbamoPUdURbKKnaSglbGoZFFOzLjgMPFcygxsMRyAMtztHUmKtfnclxOsMDdmqGmeslvsTTumcmlXZJQtjCakcVFPUMrEGvyCGpFcKSPDHjorpDwKQVolsYMwUXSUHmMbniNLjqretWkdFFnclQadzuySaDugLBSmiExzjsUZYOgaiyFtsOWHiBPhaLjtJLKUvzFrFOWQwZDoKOFDEbjdOFPDjHtiewWKpGpziBWNojBHpfAHElbmVgtRBvtwzXahihVAWlYpHPvKqYCiGIjjnDhuzYwjdRgPRPrGbBNRUBWntfzRoDaTHsJXPisNghLdffXmBkbzeUhwRWgGNBtroLNrVBHbPaGOtQSIqwHqODLdrMDZckVYIuiwyoCNHrIjiCLFehPYVncGPcswxVuAHRXmbeUztSotEyMAcPVZCUewlpctAXZAZxLUthVwuGsNnIxHGkUZbfxPIqcowbQLJWluldDeYhXDTXyoUbomDrsfCorTfoaKOGbxGRhkhjUDjTfeaONXYeBMhcahMClhMhHSMgaTPJFWVzUibuEhTvCGhJQRIEDaBJBruLMJloaIGjbgYLmpqvMMpmMizsnFsYdXZRauoFpOUSOhvhmhwERhwCHbCWIgcqsgGCFjpXuuAdRiQjUQekMzGzknwmzKDVnvOAwQBIAOoaQFbtOCKHjXgBuWwYijgpxBqeEFMWGFSABgDaTakJMCnhkCRUWYmMybZqKYLUixZwmsdGpsCDNcXknYHUibcOiBaYFvWtqrZgQlsaOGAvpeUSnDHaqiZbXQIKIPEHOyChNMLaqDRgSCEnnjaUhNlknidpOgeFKrJAxttgIeMzbNilnQStjtVaaFVAYLnFucsNRVsmhVZlmQyzrOSkmPzRerCdloiQIgLWmWVFPreBsJRDyMMAahnnefrsDtbywbDzXqwmUBlCXzSZijYeweVdvNmMeMvUiocAunrqHrYdAVRtBCPzwApIIouwZbYfMqtjDVnLVDgALuPAwyhgdMwvQZKLIDXKnjAQORaitLpslNGMPsbEoOzxglYxwmDMkrVFhueTnymlNuoOOMGHnIjFPveTdXjcIHRmTTbTiwnwIDORdWFtPhruVHPkgYfFMAFoVnPPdBUyJtKkFQcthqhpXLZTYRTjoPEUlYPmbFlscMuZjqzbBNkaylqrxZkojyTMPEgNkYEbEadLTqEjAFUpQrqHpPqhjArLOYUpWxSNyOwIlORrhtNIdgjgeHClRKSwReDdfctwNltRKvtupoJMyaZRxcnJSmMwoNncMNrMHKUjZYoKkmonuSNjsdNhXGJtzmRupIzZKbpCJoZepaTqdXLqUAXiIhjCKNFmCLVSBREGonRfWYleIJPMIVWiXHGLWRDtooXwoIiOLkqGwmAxIWGFFLBVPhNVLySTzPrmEfNkkGXluVKRERBfCZBbUBtWnnWLMYoLTOXHhILdDCkWDyHiUABfVwnCkSHnemGJuHghoIiKMviNDUOabgXxKWDMzrybOREMsMMVGiVhJQafOsDNQaLueWFTqbxYOlzztoXQzLSTjvGvEomYBNulWepwgekVrUcjlLkvuLBJYQXoFcVcgymueUMNXcrVKqAjVQUDoZpaFyVFyAVHdJeBxZVZThcRPFJrNtpyApmgUKisPAjNgflDYNpoazfBNbEKVCcYVEEmySphPjSmuwiFSmBTWlhVdsjLKPAZXNfawwJGwTmKgwRxakyfbqokOePBgvibRMQuiIfFyolxjjMKeLoLSYIWNSAoVhhWLWOggXztWSQLJTynIxAVcMYHSmsNLlPnSoVYDgLTxGnHdfBhwjSXwuSKmMvaqagZCtPkWGZBOSLJsDflEBleePRaJHenxeJGOFntdUbvKhrWtdRbbdcVKORcvlEpHlHkQvEGJKCCJryAocXohwxkUGKdnqzaWtXYEoMFXNYefwKfHzlmjFUzikdjaKVYBLSWelHcXbCcWTZkPhiAKTAZvlBFxZXtVnnmPDLuPezbrjXesHseaiAmEJdFhvSAGZSAnTRJDuPeUriRGMprxQqHXAdoVoEyqmhcEaXLjikKIlVKFhiNqmbmySgQdvyWEhoXcJQVSHxvImHyxszsduKxBDKrnpMozLvNwsDLpMhtJQqXZUrzyStjcDmgmCyCrzhjQIZJQdKhLefKSFIVYhNDnzfWWbZHAVddJoZkfgIiDWzIDONxPIeVVglUxyIYlUtJsPqXsJedWnXlplsLFMEhMKqHlllwTTuZpOaDZuLJVuSCGYHCxJgvsEXnQYBFffEZRElYbhsxOisOuqnRzZIZwYBldDcvvTdBZUgLRZseLztsWsxlnuwZynzFIUQeigsHwjNiRayoUMwxokxZByFOukLfhlRBRHkevVOTYYeXqgqXecFmtwRZaOPgqjcbfsyekPrADKOODIAgnWJraEYRTmiTfHIFvslbibPAIjVJLXbxZtKtAqpApIvSFHbWgPvkKNlxddvKYNaSxqJloGMzVkdqTSNkDPactKIFHSxopqXkjvcPjediTEKgXBokpbFJszcTeXmlLstfRvgANwNyuYUkvARbYwyZlIlXuUBZVmxfxZfKEJGutcXlwhtgmHoryijZGGejCYYgihQNeyGYBkphFLfGzQHPNWoICgsQlADUbAHkdXOwcOSDYRQFuGJouhVumbzoxaCOttEjkYhFQExaACFQKgWvLBdNrRnbEhRgqQLBtzGBrXuzNWAaaXJdhtpNSUXkLJkNwaklQRKSHfORkcHkLYYhnCWGnmLRwJfIprjnUcpQDWLNoruvGDHJsKPqxdrmoPMEvQDhVHIeleNzXKMwwJkaZafljfOWSdyAILhyleXcoFVKiKlQjoTCeGkipwfQbATvaneMcoqmTJXznlVJxnNeTLtcpibqCAIqyLNYmjFdCWeKFcHTcbvhiQtdlpMHXXYsWEqerjAJjjgupephnpeDSOKIbMeZyfziEMTQQcQYoKHqAAoxwtswJALLYgVpNtasWUXmXWKnzWrsdXDBcbCEOpHMdMhNmfimDlwBhWzlAuePAMBCLqChMlBDgYxPmCSiKCdMpGCACNiQimdakFlLxcSplDEvwargvQWhKGXhTjeThzGnXljyPhzmYranApSSYjCOtLSJPPXJwjwJCKRcHwqsvvGgGYexxxSUdEPrYuYnKioSTOJaQUMNpCOiUZnbqPJyLGoxjWExxZcpdazHtOGStpkKMBGbFXwMtzcVKrRofiByJTjPfwwEQlLVgSxlHlPcTDuvRxPlZcYjUMjQXTxhBAtxsblTptvOJIDaInWEXxFhxzGHbBcZzIDBCQJNLVcMVjGxyTzumNlWakuiiqEzitRxDNJnzRgdoEBTmddEkSmREVCEPztpDPYXykfOQMYzhbeKAesxZFqhhzhZqMbyhpjSlLkcHtWGEUeBLTlmNozYOwpwexwuIBdEjTLAtCLzyNNHjQZTwAsDsqkSoKNJhsXfonyWrARPOAOniZXHOWeryWWolKqjfkTHeLOzTLgpVcdeyVftkpVYvpZXYRLgIjcnjBsBBWrFcLZbuhuWlpRkQmxPUgCTxkWFexcUOCIHghCBxGWoTVGqWhidcrZsFQPlOAQfqNNZZiDcACmkzDsdCSnxmDjMQpBcqbyOIkSkjSdTstHCsfcjbMbNbWFmRAJfSDmCHgfDcoFJXWWDiTtxZiPVpfctblohuwbibscdFCUGUFfKzfqsSMEyCKUXzOGXjQIBVfgbgdlDlDnIswomImybYoQlOZzHOqCpBQIHPSKycbYsUdpXobyimsapvxpxLALrcpujIDOlTAxoOvePPprOESsCMkEdGChQYczedofvPSGSiijcXkfTWOydTXBQYSSLUxyoegenjMWrxTsXCcImsLNTjjVypvyaNUFDJyvFHVyHnOlPLMOEbauLKOVrlDJfpDvzCmTeaZYgzgtcbrleTKIzSddSqIDFHSoBXkwbaVmnuiTTzWDZwrJevWHZxcgqbKFektGkElrGpmJIHJRcLNfldJbNfApvGkPvAmqLugIuqDvlSaIUdvIEGqCOVSVkMmpwHXzZAsnCoLZQLJQVNApQuAhmeQxxXBNuJwXLZQjsirUxHTRotdTFKPEhfiPLGHyzhTRNpLglwHfbRxFsytHilgaSgBEwNiibsTWiJfmuzzjvcwHnzdKpXLUdMhACxejskELPdtLLjqHGfUfICtXeRkQLgUMcCtXesUvUpWeNAGkQwyohAbTayEJdrXpObSVzwOWTvQPZdzkUyfKaWPBMGACVLdkISkLsgYftPxwYbZJnhATVqlVFImFpBBMIqcrBDGqDJuYkfBZOOvVLHJZBKJoMAuUrZrEAUhpMLHpKZQHgLiVnEnHChkfdrfLNsBZnfnAcjdLaafilusegTKnfdRuGKIApmKvUGrYckEtRuEmpojszsgubpCxqBRxbPOBrZDdVaMQjPVktpHmOtOoVPaIAffHAQwNSkgkmRywffVieTomFPleEOqeZFcbWXzLXxkTPRSyYwZcaxpFXlfRmfaVkBeBocTCPnaAvwEcWMmBAHgyRipBXGAmcFzbctZnwBGYHoKdzpTHEZcfBoKDMrhoTtMiCliqZXNsanxtTuGWUSgURPKGNdyIenCKFTBYYVTSaUXDvlOrueCstQGpueroAZWyqlBkmyUcwSJlnPYrUFDwWnfJejnZxlqHUqhYWFKDhPmPiXyoViSnmNrxYfxkFeLcTSxNveZMemutsFhCDmEMXNwKvUtGfrFTZrBRqJvTYjhRBmQDnuGylIRDYEJgjTPoAMxbBgpRYOqammLrsjDsfqdHSqHHuzeQnBTXuBfJQUsbWlWmyEtaLZRvSWsSaAsLYQnNKkbxBCqtYOMDvoXEydcJHMsYsFKorIjxlKSttUZfBXvksgOrKrilBzZHOiMTQcesxehzJUVIMHhEBKjZsgJFyZQkfMlGCBPVQQhJAjmDtRhXKQANxQwWzEEDghoDpSDdSGfZtXZzGrdoIKldgRwugHomVLCJvNIYSUYVaSaHJREtHQlEOaEWVoBsRhxLdQQsBGFTjfqzfYWtKsAyDgYVZuHpEplmorcXzgBXAcMEMitiDXcJjwxzolkrLEhLNMNsOQXuZHlFSBMsJtoXQBrayfiQFhgsdTYZVynlLQLpoZiEwryPciYVIFlsPBRrQVvBhAyXbXzFWswyzbUYduTMiPhzlfXSHOrRHtNwkqteIsapEJuHqUzWHtJVovOqgcumzSYStXUyRyZfZSbgkAbdvNmVMXxZGJXQTQLeYVUOdxbWfytNnBZvbvDkeopQgyprPquFjeWQqXeIvbbvVActTBJPdCclEZZpiGzasNLZLVsYRLUjPODEAjNbcRAywKjKapUzRnfoCwFXxcJThoVHFMRKyYEpORBfuzIXXPBbiOgtCxUEEDuJLtYcmGljaMYwmrmzNRsvNDtSfalyRLoaBiipSzupMENjGPdqgLjTfagHsFVSeNNCtQLQMGYrSIGYSPcaCzXSazXkzDggUaSlsqtPBuFMzRqfiProjOWDnEvzDgjqohQjBYGNdYGZPLaMFVDCREkRCWRbaubZntpWNzzKEvhrfwolOKgWlGLISzuyOcdBiPmeycareSLCbpYRPwJlHMVpmSPATczZXZxxgVxlSqTJMZSzsKoOvDqgXhcoSaOdAYniHcPrjPBfRGTfdAcHLXFVQkMTnQIeJNBcaXUOhysaRwAaDLhJbQXGQjrjFjgdDViURgDxhQVapxqJpEAWUTqGqQBLoORelMuPBUnKqHpYVpOFjQzOGXMBSVKJaVpQychRtxEHaudkjNBuyHpRKbFdCuixXzQttQCfXYZXGyzCpcpFSydMqKkWRhdUnyHbGGnUzfCpWsTkaHVhjEXtzGtWAIBiFmYryxqYfyWMfYZCYyEnsUhonQhmOdepcjIIZglWYsnStvKFCpzlGkOPDVhPhxVcHjwbVpaDKdqYqHcrHMxrfJnzGRAjiSlAYgIWWjcJPRVCpvqvpjgprRqaCCPreLaDJwwhXhWecXivCVUNCkKAmdGEmEmzucvlBScyQDtILMmKnyXtRUSBmTjQAmzyOdxaOJQaxaTwDqCuVSeiHBFwhrSUgLekHauHOqsFOipSqATWwGbVXUGdOvDLQWXFGpiqPLSqilEfMcVgqqCMcmvecdruClkRHLrKYgBynimgscaIuLSiEvapZVvNEZlkeyIpraJdRyZEPMyUsTWVMZNGJEDozQDqcBgtkoQQKjhhuyOYhlgvnMHmDXITeScLabpvSOtrutWauHRTrjYKsTHekWmlakaCBSSuWGEHuHqIuTCUpTBgLyKPskWOqOzuzVYVRVScUiFImvnhSiGjajUptynimXaUzGvdYWuiysxfVHAcFfMWkhTNokHKKMyvJVYRLRjdgTxpuWnFdMaqzxSwkMuakmsOWynQoriTNhrAnkBVzUBBspIcVqvczJXKEYZkoHPCKxBMcERxcWKFHHkZgspPLpgyArXuEoSetrXdJxfQYeySOBoqWGSjHtBdtzZfsODjNXPuEcSJiepexPQYrRClclKfLpuRyIUoBFVQOyHsWPRCaTlLOcwbFTqfadFYfvmcRtZeDuFFyQYoUYguBcwYAJQnaIBXhUsxqBQPhcpEgixlnPscPUPdQmPZVxMvKnUQwPkVMWEbkdOWXrEFrsEqEKmhzCLwMgGFXfWVSTXzvaPEeZVxcSPyeahVTnubiMJeLDHISYxdKiqFbSozYfLHUyOsyWxQxIKrmupaGowsiqpwYOSlezmnWBlcZmPcQIKPnWLpGxFFHcMxmtVwzdvftKkpeIEzsFqpCSBpMgzkRSGSrHSMFbIwdPdwhtAeqbOaAUgllhWewkRwKJGmEIPQeevjriYSIPLOkYeLkaUuXAXtUXAorWWeHVjGkzKxJqdJpqVUawsTOmsYPoAJGFmHoAbUGjLxkEiUvWyZaQOuepmkaJUAqxXkDaUUAhqmudMMKPwIyZDVClUPWQnybOmDCJirDbeBZUDnELeVbPDhzfXauAlcMuOtZizsOwPboCmuqGjLhthEJyUDzjbLJRrlKQbkzyqJUTMoaKOkgWuCIFEAINiSuKdEvpiVbDAaEHoUIrOPfNMXsHyBSumpVuXAGWpxdcRANkvDZgfBfJShOTxKNGLZTOfDUeJjGHLFUzXIkGPBdMnzJhAjCewYoBUkWSAfLuVgLccZLvXKZIwqmWnmsLjzwHOPRgsryUVTbpdIRpsoBSARBniYPQBaIIPpLqqStISARnWqodOmtnHWtBEFyddfHosHWMXKJoVWAsndjrvtQvOSYsmDdgectjWrYsJXZZLealrUWoYHjTPuNehwmiDuwNjEtaINjcporzWMWNQnUeuaSzlfUNbWoLSVOTXDkskeSznmxWMdTfWnNEAgWvOhuLRmJHeQFGlcgZqTrwHbtJMwvjFhVFEBwysilFVzICCIQapyWdTovzPxiDULRQsSJQwyPsidUkhYlDTgOPxewzoeMjRrsmvnGFvWNMPyopMzvoEDOGeRXPqHvjIeRkJJUZalXjayIWaeRksWeSofZyqnNUuOkUpxENZoCKFjTXbEcCrfepHkCRAMCqBUqmESNlPHansPeVasteyavQuBGeDBDAeuSxwTUagYRRdWynObIaoQsewJmkhaUOiAoRYAndPnPPpuEbZWEQRLAFeMaQYpvSEyFSWgsQOPhNsqLECpCQIMIoMvdCvtInzTCGTUffqqZrTbzlRltRIluJPwGsohffCLeOFByGmwxdZpWrXUMVmndqjYwagHLZFnllcUhCuoUFtZhMCyUMxzbRpHaugSHTuskHSKAdqtpMANiErqLMczUCrMhlujXlQTwhXJgfzEexcrgGlNesQsipQhsQRoxmEmhMonimWMxIBcMsCrbahvGjDZfOnMsPxsemrQUKipKHfIRQuxmSpljUePcsqPzARDaTUGdZICamPZLvDQpPRkyzlNHqdeZathMDJLomjjuQLtzQcVfhBMdwBEMQgkkFvTFgBPYWeXpOlAvhovfatAEdMTqtUXgjlZLIEIjLHzwMqVcxNLKgtPGZAlYlsvyaSQeNzavyVnrkOLPmyKLgDeeiIMRkogMcQKyThyVAIbJjNOMSGKLeymZbrXOvNtavFwNUodQoummjPrdkTWsZSqgcvaDkvNdWCpfxiMEKrCqZmnRoScuWPXCtNCJOhdaymhIzJwankhGDTssNCmLOszAYjEHkEfOaBbONECrwhBKxxUYkGwCnhKUlGEAvmyEGnUzCdPnwzDbEVSgoRaDBBzbIFKHjDUpDKECqXOiTPeEhoPGaAGgzYFXXLlrDMoJSGFxucDvdEVfRUTVLScdekuStLTVqnSOKHxwrexdTGsaSDfBUuFejcqQCpkglCEPAIXbdYskbkWHuZrnKMblAXzYYFPXNGuzENEdrcEDGAhcqtzucCPXqozgJyjqvrpnnBxIcmpxHysROVbnEFRztbFnXAiWatqgyeNzTwRURmPrUJrjPjlpKlPxskYIyTCYDQNuWAokvJFMmLRnwxXtdsRXNjwyohItoLRwfyyycYRSPygBggqDqQCzvSdIyEDPGxjaRYIkzJATcvMQggzVVjQQmBOzytbehgQOpYwcJcuIpCWsBIXakEyzzdgKUlmzAbJeKpFWktXPDpgQJIxrLNicuxujAQIXdCrIiXBbFRugIydcgMjNERIGMIScZTnopawopqxFHVErkZsUYEfCcFlVnuLjlGCpGBDLZwQHkTkGHiDhoHhNXZIqMKZKoemAqCqghXidrklSJmKJVEgkIOXbhWgbmPuktxGMecIzUsTdhJtpAatuTHPSUDejCpWpRtTWUcDZliBWWOALeMJWsJAMBBcgmaTXCbDXSDkmbegRdNwPsFnaZRmKoOGRcTCAHLWETglZktDGOiRQIWFMcBPTmTuzJtHBAAXjeEvFdQGbXFOcQdvsnrsVNlwukrrjsjTpoRaFBzOXimDfEadRuepvqXSgjtfikcBzfLwqvkxhuhGkVGzVzNCsIyJaHnzIreWCXAmlCmaCsHgNpbjKpMsRxtYKZWBDsaiSGRUzXJOASLbdwKtKFALIDgqyiMYwvoIbPGFfyRguMoXXlxXschjXthggcCdHgdCrlJOjkRAXIQGMpmMgemldQYHUcMoGirRvGAhgIxavBitahXuvvQqiyGORnVqXzameyRzrhpdgzEZdFsoOMmhGLGkwMFMVdQdirwPsrCOJacRoLfOaWoGWiCKJhVbZncvOMHZPiaXpyCfzWTFzsZCNsyaAneBeYqWCewQnTSFIMKFAAUgjAqfxhcsYCajUsxyzzGiQfobxSPvZJesqaybbqnAcEfmHrqLZMttWjqYDXWeakinDpURafKfSnyGlpDFvDsTLhdayenPkZwMhZTQCDmPrNTyWOdkRJDpVtmLDFrnmevBJdVsrGumgqWKbiCspayjmQtoquhUsgqKhpjzkEhLaUNmmKpZrfXhxrjTOWIeoVbxTGOZDmkKSGgoOkuWhNHIGpvspqJCPHmiSuWvDEsfjdoLZlDwzsFYTbwKwPEUJnNEoDtNcfGrugXHmDdpkGVKouPrjwszeiBvPRCieHdUMuGTtgsaDEOJxvspYbOThgYLkPBNgKXsFtKepKqUgjgXcbcFtWFzLXCVUYAruHvJRdVNLxqruGsueEoDrbOJtpWayyxeypggYfIQHByNqhcTncFtaJrnHILDXrqvtPcqqFyMNoNiBZxcaMNKpfuUbynfYDPMddauCGUmseEhiYcflJURdLhgMfaLeyjeysxSkhtASHJPdyAzGpvsYiNQhJBCkfxVAZIITxcuieEkvodKMzxEocpmiSYKHnbKubaAtVSYzzlAioAMgeQELoCYFKYekVLSpssyhGdgGgkyxqCLEKyHoAcwrNOriUbWVeUttmmMYbifNZyFfcFhICgzpfZJvSeAoMvmbjuSIrQxcCSyWqclPnAeVCweVoNMmCdQloHUHuZkuVCTiJECEhvJhKdDEhXRSgbQPMvHTBUFGGcAUWRPWxjsVoWVCNzlyDmwMdbuvpHaIfamjtIpAFhznxqdIVFhEeFppJBiiluicNTFVNavnpaZgjFzBDsloVPllScsVrYVBYPWcbeATAPbJQefKxBHGIaFMuWWbZRRMfycPvoCddRgEvTWVfRdvqmKeENDIUdQqFNjkWZuUvCBrcQCjyJGPZNmDWNJRKFANNpsjHaldYkFsBgmABHyndWXysBEmbWTZTYzYaXqhVmlxhgipfvCADNPdyxmPhqvOhwOiOgOTSLzFcElYUMnrwTbvvgpxgnmNgryRYHgxNTwkbfUwFUuOvfaBumceSTsiDifqlsVFjHBWBpLUerQoCFwKSuglaZAFlQcLWxPjilVrZPDgJDkyRKMZiBEspuCxHtgiHNBMyhwqvjocVWujoigCmFhHneQzHpmznDgIYxqPXzkxwuQRuzJigdqPtqSOGFbFJdLEOmIPdBYXFepkJFsadIzctwfwhdHyBogbXMXhuFVSfrUckFdhkFOwNzEiNMrLTOFBLYcReLNXWThczVgmbkBdxVBQchxPWIrJEPfrcWhKBUFbULXYspIdwkzTCSOCuHbCaJIfyOBAAVekTcNPsWHHTZuehKnwkjajzsFpfRXAhbwekbFoPWLblgOPpRATOuvAZCZsiGqkTYLkeoRtkCNKdbBSvSClLarxHaADpkvNAluVfEQLBfVQLQoeQkuRmzSyYuZliLhbDloYbKFTgZbKBpwUzYpvhoRjRmKbMRpxVRMlmuKWRVmtekISWRkWCKSyMnFnkLJHWgUImaScIGaQiCRYaCuDOEljbzcagXcBwoBCGsiTquTLSEUtaitdFvbTISftnWRsFtCdifWOIldcnurQuVHjQsjWftxmjpAZsclvAiimKjfHthBQJaroAPmPQfaoIMqLfjGSmzBXhesPRjmtwemdJpNvnpnYxJVzdxzjkFabkMbAlKYYUHRsGPgFcGwZVwbWuPyMqhbbEsFEVYmyIMnOpwZSAWJzRDADuOGQVdKYyJxIbbBLJgudNieCGrzzzuThcDZiPMqwarmLrnIXtjplWiBXLOwgxnCVWRQShxIWaGEykbWnvnCFWuGowJEvNTaXFUxHEDPLwZlHDMtDhSOQvLIcXYfbhZmEMsZNWJPECxbqtWfSapqqAMbPwRyrAMrSCJWjHLIOScLLJeqLGoeEedVQxYIAITOjWJIyUFQlKRxRisqYoqTZQUjwexbFJNpuVeqhjvkCeFHFOndRFTxmNThBWuTVNbmndxnWsqcWWLYVcFXIuFqfUuzkhQFQbVMapDbjKPCEVOZMyKvicYKEksybGUeSIRVuijBPmPBMJosddgkBsrQmIKrXwosSWqhOgcCbJgHNPnorUhqwQZyiQDYUpaXSUTFwdVKpuTFDtYLiETNtDFqkpGPmtloDCGOeyomGxTksSnWzmheIIsvXKibWzJDlgrggOLdxtWkQMJkIFOqtcuLnSNZhbDVeApHzAuYpJxfYQrFYFJIvsWEtOXteCmkybhWwKwwkvZKHPGoJOmuayGpjPVMMTiVVOpzfyIPRRsZRKZvNkiQYRTuUZjqlrmpjEIypzWycxJVSLIIGYTupICNMhwmoHkFRThIfAuvlfvMLMAsLNyLNlpMmbjlebbJyUJdPLrwxDUwHRvMdhBVsRzOJkQpUVnzlErhxfcpEAVtXNlmlcOuMRyHNGafsTsSYUWKKBFxxziFHgfXQIqGRTnUBPmKVlcXvnffnYmGlpkBYsQGgHquJFrXrpUCuoZNRczlggUPbqvRAVigtqAjhBoAjznrRAevIFpgONuBnkiNYVQHoqLgWItMxqMHmabTHAmqCrIrsLiVDCFWgpdpSxcJWLqVIYMrKDjoHLYxLTXNwbQMhwsLDQbtEEpjUJvJpOcOxjJTuMulBXdeKOdErocUCLtWTesMwiXTLgArdfgNolmUJMqIxaGPvQFaOTNofbQRZQTToMbaHuLkBtVawcLkKMEqpmjIyYMtdZnjypCVBIbCZJmkpZjmQpKfFFEWVRrHfnbMRxjSIGKaeTRejCEcxzsZrWWvQlkPYSqBRytJxxrEFJuaAZaYuNylORwySvPKfdOkAyFDsEBdhlhHGteSQLBvUeyvsjsakchYFYcjpEceOcyeKYXbosZUEOJXGBIAWEnRPSARyzrRlNRHvZPFjMEanyHoetHsmFoXNtIXgckMDHdLGOvpvkhaipcUrrCCrQUditZAzeUPuhTildZuWZmfNyzVEEAfAogYUtdQglxQuNwERadsxmyamkrUuQzYiNAlHTXqlDhgwATfbutplOJpPhUAiAgeOLLuxQAqSjdEBZfKNObClWbVTRStOIFPVCjnUwsSWOCjgxvjSCybQfGRBjZATdjnsjVPARXfsuABAMasAFPPAuJexejiUteYEhmsdnkedaYjQAlGvDbyVDFGeYawSxsJmnLdQzETNUCsbMQuFeqTGXGiFoLMNTTOehLjIbmKTZdubXnzeoXPvUtpbsLQhmYlryzjqZwvowsrgsCTISxEkUVaXUYqkPjcUwiXWudTOPombPjAPBilTxarzhIKVcuqvdrlaxDRJNYmKNpEqtwRiZQORmQaotEEnrjufokrOZLmxQrUQqncAhxTOAZoNvgOOzIFRsEamdfunzcMmDzZbZvEBPLjZPZKXIxSwLZdCIAbyRAAqTGadPtyqGugIbNasKGjOhDxYNTNmqsuFdGLFotrFzpeJOfSUNWqAbWuWAwtsCeDvpIltuOhLPTPAQioHwUZOTIWbiKsSjgbWtUvgRLXPyNpqMoncrjNVmFJtchVnYlLqmXfZodrzYqksXThldgFkRyYBuhiftXNrbHgJReLwCKNsOpTLWvQRYfDkzSuKlNWvstHjqiriBtgtwEXMCHvIzZpuENNPuJmeNxgUwWcNRiusuuITNIYPCUjUfGcKuVvoKhkwUeKDhuqyWQEGJVmVoolbJbadXJZbneWtFqWiUwdqQhwYNNzhBLwDOfHecIrVVweXKLvDQzpKWkNbLQTJGcNUGkCWNqMHeKGpFzUHXIfSSTWFutRRIpQdsLLyRqFuIVUrGTTlWKWuAyrvVNVNLabjvCgzHgmZHDTnCqcUwItGIBLJajoGSlzNlfUrEBGaxCVXBNmrqEtaMecvPvdyQjQhauWFktrHfLEDGohjgJXEMFQBMfYphDcAoooGzmHRuTgKwGZHWfRjyccEHtCaRoikwckaefCIxgbxEVtrjXhhTLsBrJPFrCEhiNbrbCxamGIdAkYzDLSGpDSSVKXSpLTFEEauGgJMiNlkvMvsKXygWQnXJKFhkxuHjAUIzDaYOvNdIbcLNRvXLHxgEZiuCcxozUGHuRkwMKqsmlCWdRUNJHHrjRwpnPaKaftlAWtmzlVZajVopDhbjSnqiojLIcOGVDiBYFZqtKfpvNPwFblfxgSNnuMNKrdOfHmEiwdwhBOlRvQxCWbckbTyrGBdbSDzJBGPVowYhYFZCbTEpYMPhzqPRLYSWzQedqqfmugDBiplLzZjwZEmtpSxSkwLgKEOWLoPwmtFILNVxMZGVxcQuWFPfSEzKNOykUZVcSfypOZfifDkvZdWDfJIRQEgFTAfLiwAgUXYGTbzAnPzbZJuNRaWgKmtFeprzSOeGveiOKiuvZNNQvPbUnqfpufBQtqiesLwAmbslOmhmldLkDlrKFomYxMHifTcWUxsOZqrHzpTDMPUlwFeopqmDrGqoDuVdWYgvYoBpMyoaOuKvxQzshrTDvihrwYzQpEqbVNLKjBBthvBsGuAfCdKATbyvNyDXnwNmxxrBPtdHRnUdCmkcJjYSsdICebZsCkIQWJWCZpGkPYxDxyVMKmduGMRTfskicamFwutybFccTsdyzOlflXNDLxkskjrljSZktsFbMZWoXvXPZiojSMvBOBrVsybQcIWiYAYozOzluCMYSKYDXkTHrNmXjvZVOdsaJuXEDuaquwneXfhxjcaEFTafrDvQnkRZAvccrqYplJvGgZjkKRRIikpJWBHTboddDiDQzQzJayUQYMJkSUZhKyugxZdzKRGlqEFSqCoGwyFWGovjHDmifkWbKmAjeZXihbHzRAhJtTqEsjBZYUfflmcMnCIWwgoxJnDjdxecHUqDQpNCBjYSmedXranAMlmhJBNqqusHuYGwqZXZTMrNCvKLKDgnqOGDIBzNAjqPeyucjcIhlPHAXVtEjGPLfZkCPngYCgkFWbXJyXEICgDMdexdvfeAhVqLcnsUGGDMmQysWivgcELccBifVdBzjfaQwwZpRvrNEbjyCCBLtKakynaCtCeYWAmWCtmGlfmZdCVHbKJVBIjQKhpKoGJEaYFHuGmlAMXVXYKuReITapsGbzjopBLbbgoJbtwwbtMjQotRuMmzLgEMiLrqZKbowaDQpHaJJFHybiygfWTkZuCtkUAveWLDQWVObCKpmTIlpfvKTlBOdZjWBUKPDqHUFvEsawhjBkVIHWcpjeVOCfGKrRoSFAXEOFkrBXWOVkIizgDckcoOrmesiEFLxenJVluBmlSjGdOWMDztGzdOXGZuoRQklzPUaMkeNHvbzVFPeEZKLvrdrgzKXAkdxjHfrUwbCcLpSGDrUBRLyjSQMkyyILKncBqcRAcvVNkZiHuYVkQjZTUpHXlBTotoTuogFHUMykndavbGXKRSrCmBBIaxmXNxuUAeNiPehRLLSfkZuFxcThExFURBwHuicBGaDLOCYhVhTnhxKfhOloXPHFBcDBLsDajiskvgvHkkOPZtmPgkOmiDKtamICjMkgWlLCNCiMBbIbkHmnpLDbfAzIGWXoVdcrxFFQeVluqsOrSmOaoPtWlTYzIiAIrfIRiXKWUBcRjEPFAnRRTCjdVxgUdkxZDbQdSUIYsBAwiVZYUBZRwlvYVPKdiXaAEkDWdiGTHSnGxSXWjHKpAKtLpqNDiCyztwUxNXcAUiQWzzOFDhTfeYSRLrwSdCRcYOqlNFsrFLwKczHYIzxAwnmdlyuQNCBPFXuBHoBuUzRruCGnThEFlQkpiPIbgKgTTaTzPhRgKzSnoJPVDWqerVjabgUgcTeUZdlPnCjkpFEItInOGJwPhjsuOmbCgkOsSjlYIEPmZqLQKexyGtJjkBrGyfIEzKlnsgTdlNXOBnSZxmKHqLnenuRHDjjuRhiWMsNbPObkdERwxgijfKMkAjehSBXilGoOFiNViySqKfvobmQmaLwystCerfnKieuwRyEBmcghyDSudHAABLEcbIrNzkhfPWOOIsDbDKtWDpvRmCDZRvMXXPwatEvDQRZpqmuyLTYnvDjgLDOZjzFcYVsMelGqepuWfMMhKAwqJLVbzkTogbmaputsKYAhGGTHXxIBPKwvVhjxEiYaspmMChglvdmoUjPXQcCpBapFsjabZxuDraCGDcobpWlCUfujMCQaYZNisbrugYuLIjqLYZzjPZyPBbCwvSISnHJUNWRCBhFsXihAifHtIMGeRiZhDVoMfNbcgAITBikkShvFUbXDBMtUkMpHcdtyrzoqhEUxsUbtIqCyOQNhwoBJFJsNGmpXAEpIJRaSgVmeahCOuiVMtXfkzhzPJxfbWwtHhnESzGAAGofQiLpoetqIHmgLbvHHSwgDVesZJssVoejzkNazkVLwMmhyqOHhllsjvzZRSWZPZYzInSjAAUzQZQTbLKIExHWKjlNchVrgbqwpWlhBIpkROfQKRdxqkgDmZackZbIyTGiZTgnsdfNfArCvTIHhWWYEupUshfWzZBAodtMuwoMuZiZksZsqjPvjVubFmBexRVSJyQLaWCBTBKDUAngDzqhaoCqEVvJtPJcfMtmViYBsOOwrgXXTwDVXUKndyVeMOmjvnCtelPpJExPjZKfjvORekwksAMLPpGbToesaIMpSWkjmuBuloHDxcHriUkRXhAjywnEnfnsQaDIWVwTYhgPrRBLtNemQxlBTdwmbqwWTJDljWumyGHLNQRWCZATUSuLHOrPhGydlGXQVHsRtAfcOwdmXHPQBAldmCDkRMAFpEeKUZiyfwoRqCHJktvIYMUWXVJoUVtHRpQaSSwSexeZkobsszAgRGWBtBFrDxEYEMRhvvJJYiihEYdBfhJjqKZkkeqrujWioXlxLfclFZchdauHLHCfYVzYSpiwlOElsppZYGZcZEbZxNqMDmAMqHJOISQiVUKAlSTpRNQAkQwtfNzhdKuoBKjxJbfuWXQHLOpOCWkMzsplcioZIxVrudDeHburcOMPXGPWrerWpFaINJdFWDtrWhxIYJrducTqKmFRgUIsDgGyNTnsnjExsmBHMnkphMgJwcUrEZXETxkFQSqRNZAmwKBijkrYmgWSRHAzKKbEOYqcKNDoeCTxuxrhwVxFUqeyJErePmwGomutOVAUOBuQdzSOXknFohgIGZFzeLSHSeIiBFBtrlUIZjYNDzVJEOvBRkslBNdZvIQjcgHDnZSVIeXYyffRFxyEHHNzhvBAPJAMNUXonmNZnOwRqqLIoKFeqFqvSlwIBEzGZLdnglHuLMJVNXNyDIUbOcjsfUBuvwsEopbpgElfleGBLsdIuURtRkQpvGTwULyfMwIpYhGxxlfcmEGbKwnGEWkqvWrlfMxeJsZkSxOlqlRxaHgHaMmZrgpikkheuMaPBZiQqJDRHdeBPZVoFcYsJiveUsdPXmyexqNmYByukWNQRfyGYHkVJzhLSXaJQIkcnnUpNUJJFdlhnfsSZtTiOGYauntcQpoaOugVjsFGSBNlLDysZQYwEFoBPlneYLypIQixeHJxQcmAKVjxMjCLsUZpxACRyDdqyTpqXdrTWeriVcxtAxSSPwuOXZJSOHLQbWRzSMLRicToccLkfFSJAEkXFlakGKpcPOckxzVaylymqxNYUHFaOgvcvICNqvRrBaRrTDntQvrVMekEpyzgjvOfDzYEERnshlTgBNpeRQZTGsdcKnzYjBjbrVvdEoeQpVCOzjHxayLqsSwHPBpvAVCXaUPqYKXrPuEULkfICRHBRHRWFtZKAtiTWmNuPZhMGVOQPONDIUCppsscixwORJGikkCUuNFHxCPNzKmtrxJNCLVrbryIbZVjvqsZFwkXSjkVhgEjRoiCddYRlBYRXqiYawOVlrdfaNKFYkIlnyzYbdXSNSvdKkuhXmvlEWkRUpavKhtAmdSzaxCNsGyKGvqhadlpCKprBdNwnnufydCqeAbHzmYxmdQEbSwYauWQqfDRKDurIdkdASlFZKqxWnYrKSDqmJtYyjkQtpfCCxnvQYGByvdLBJJUXrjpxJvIFlLCoMrqvNAceEPwgnWEjEwQNUqLjijDMeSlgOgqLXcNsOAqYFvpivlJGXoxAvKxAgydtkBMEYqrQCclVDAisBBtoAxaViDkYiGbHDRysVZLqvfKrlhrYJTSCOJIkatXsZWdVGeRIssPWoanspEOqDyuuyxvdZrFRNZkKzxGrwXBpPysHYfJxHreYSTrtluKHgWqrMFJonTrieNvVnpcgWPEUvyHpHdxneeYeAqIbPtvSlmCKBSQBjHjcbbMPUIONRTZePoLpzFXkdSiFWRutjKsSwMRINJdxpRBEycaLzZkPKerZtLRkgrHcNJFPfydGIViLFrPBrSFayFUQIRgjPqnLQWRUXDoDkCsDOezGHqaUrtpKOKfSVBKunQpkdowWakxsXeqKuOmaAclVIDzDuVKDRCWYEntAYObXkRccdIevypgQPwJAOVEFkUjSWFdEmgOAHpkvTvUwUZxwAffjPlQSsntSSwYeGzBKuYZyMMVsMxBzhpMAUevVgXkpAKLbpCtIuNUcMlmKWPnrIFrgIbaBqsDuLqwDQpwzlzrxmpAXAbEwFcNIMDbVngBpIvtDRaetiCUMMKIcbWANekdERVCGYBVPRqtSnknMNIKSVIXjQtnlkSoAGwCJgAzEIdFqOvOVeckuNYEwxvFlREYfUQrIhAKVYEjvkHLjnotFpgvFfAeJEUfLDSnUSWPlZObTqTixHjCzTwwrIGKPmETzeCpDqYonYGTxEDdVwZzKAkxqtwpbQiqCyBsJXzHxanIGgvrrDmAToOusPJKgeWEYsUhgcsuvbumeicJhGuMObULjiFBxXxDFIfiWyYDHSEOtBTXJHsaldfvVNEezaZjZqpydFVOOfBYjziUZWgiofpSLVMDApsVaetMEQhwVsEeAhgkVDbajZzQHhemgnkOpqIAAwSJVHBTNNWRZGpQJIlmiSpGHkxkvOzDAxydgKxrwxLceBfvQxKcjLomvITNiiOWlBQoPVOFLOyIaFFbrOaAcMqUJyYUSNuVwEnDUuKZkcDBFrgsxkgaVnfXmsTDdQJMkQptOFEmRzwgJYoKZSOWWckQhdTkkSkJPTIbgrFDlYsnpZeSrEsijGZWrEKNHXWvuHSdNgDJaJFDjGNjDsZmstHfvFHGEhiQcDyKIgQBjZnPutKbWiKzVYyuoGjGlJtoXAFeisvnqktOOHRiyyOGqWbtqRNeCdBeqidvPuOEoqdcLEXhCGwIeEAvLiRsiCNqDUjwFKbOjKyhvoxYPoSMQnedgUDixLmtQJXyoEUEhapPVfIbaLfIhnmbWvdHfJAhYpJjnvlhgQYUvotYAJFydFYBvJWCSdpiLHTQGUPUfcDOnoTgKoQsgFjMYNRhSFjdstlautzSEXhdadCHNHLGoIrXMtnaIvgtelFvSoxzukUOlpfzaewBwpmDrxyADjYOJMByFfVtkEMLsXFPcKEwuJQQVFbjjSeWttXniMUYfXdKxEUbxaZBPyDCBdSoJfRCkWfDxTvuMNCXdojRRBZteOeQeOgGjyJfZrNyccdGSVTGipWPROqSqqKQbVFeLOrYrVweZgpkNjniWTjizGrXCJTHKhSSzTAcxWRxWeGuBgaoKQjKOekRodknoEzqcsgksgXKRpgNGQWgZCtYwJkgQrWeFVrRBiOkemLbTjfUScotpnSYamHOJlCqHQimFPTamoqxZkUwGjHxrRGFYedYbzCNIhmjOVcRkcFfzuSLsEkfCHBkfLQNQXxNVtrLVifeHTGBaixQYelkYAJctBICWwwANqKeDgZseVSUvwOEClVwzMcPqKuXAtIhRqCSVwCEVgHsJrldpQeQDTvQhDWerctjjPWBHByZCLPdgvnngVCaDtZmpGfSZFMjKRjfvmAfviqNWJvhEWBhHUaWSUBmnQHZJiQjsLOSqXWYnXGBsIdwudTGivgfXWoBOPmynsMRfJpvpSwgHVwLWkcTuNHRdfNpzyCmDbXiLQLgJJfsbXwfILLctGTliltasreTFTRTnxYZORrcwPbmTgcCRVVVWydbmkXfwAEnrhiZRXQADFYhCdNPQalYaYiSXFcJxZUapgJIWevDymlvVaXASOvYdpmHGqdpASRJxqaxsZPOSwIyBbiGhkHVlKExKeDKXzWhCUAKczouwGdEQNPxnJTuzFKNCOYudiMBrMINUGpOYMLZKsaLtnaBcLKfSUXNXNNGrEkeUfwnaFCskumQGYvfchGXxSHKdMLCRPILeDNEvdggGZBrxzJRaTaTxftyJgZUeNXZyyWVCZyXBHmMWpyjnIslKGTbuNaKAKUZMKQkarXUkBEFLMHKAdthzAyflxZBRvaQwWbKuwZulJmuJHOmISpAbLOtDoZTpCRaDsUmGnuuGOIEiPCbiVSrFupIQIILszzABKJYNXzqNQQYuDoexwZJlDwRJGQbyMRmQmJXPTTiABqdbIftTBUjJrZAkTdDUdxyEQsSOwjZgDlYuLntNayhzYhOhmLxEBVJHoDJhgKFIDCBEbtQiNuCqzaaXOljchFsPzXwtxbjgJTgvglRpCYTxssFkUYipYFEEezEBsPszMgPtpuXafaQyuuvVuGsuXwhrcyaWBxcvChdmscKPmLXCGUgsGvCMcFDzrigioLPorbUxcHQxkQtWrxkwSIKzQaAoqrvjwxlieYpTzNOalXbslBtQMwNlvZRNKlueUKFJmRkJTvHvTwSOoybRUMvvBUdCyUsiusfNrvoPXdIXeApwrAYXWbHMwjkvPXgwjUyHQSEpNnFFLuxBcQoMoKSXutHZKnHgknWfGogHZfGoYpsSmJBJmBKYwDsyRhRqNCfFcMjNHqZiOwRgJVCEVrgrGqiIHWHGqJxDCQHOROkMcDnzqaUBUBoogSyJDotntiOJJJWYQrtcVxncmGUvfbZwHeoYMhzeKVKjNfedEUTZqFrgTwHxEfODJXipdsrLznBfiQWITFJQGOcGKygWtVdgNhTnHCrsVWgZuIXiSGLEqKJaukJwmozeJqORDvsLNdevPoXZWPnzYnDyoTiutLMzdSZJIbUlWVGGgBrzEpJGUQJsZKHPBxleTVHiUBEKlQXVWwlrMfhiHwsnAlQQcGoCqNArxvgTNtvHhWlEtGzxDWyPsLGwiXqnVPzgMHnihAsjClEDYRnhTBnXuhIHzYyEZrhjzNMvlKbjhukEAeISJjSxJbzpwtwSEPQagZRlXIWbGMgGGeUrScNoDusnNFnGrYVsBdrHNGzWMlUjqSPRYXfYPhYkUxJNnZbNLrxTAndAeTRkvMIlOHjJlMSoiDRNOeuBuxFQfKedMSLmSvosklTxCEtJZRqExgxQHOdLHJXTxnousNRVGRklMyvvHfPqOUkXwJKxdgyoeURPQZHxpzoJJUSZzsBoCNpHvyKeehoaYLvsiDCSzntHNUvepVrBCNvbnEcJgHPSpmjzFIvkIVBZcbrBjKEhLHYRjhuhgxOXqecJAQDNGvyhqVzquXApzbdhrhEzgmWhKuDGCTKsHIuervOMfXLJVWutvHxfvoVTigPCpOYRJZEeZkGKSHnZgxqARarslXwvyzXLYTirEMckywmYUpGTnFjMexzQPqeyorbARAYRkNmmKLEqAHaVbtEnAtVkDWCrdiqwBkclWoPngAmmRPFXRePMSpHOBSKadGOdRosvFARnEKWUDBTxgsYVCNtjopmAaFlEuaWoZsgLKOreqgZSaPswGtKUIBKKdlLiZoHxqRJVLxOnKZJkNXqGhyysBkgQOWsiBTSZyXieiBNeKEsDoZcyYmkAucbdEddJrcPoXVteEUDAQQjlxwqYiWdYTLjDyiEuRuLGibxOWVfEEJgbWmECyMIHjPqUOtBtnoWPBXwIknFEkMULcjrvOJAXjIsHrlNfOHsMBLWIPpUYraApzMEYHpaSpaHYruZEovKjUGXbUoqYALxIgIfRMwXNGglJGgqiUYDwrsZMYUmUqlhBURqWeLbilRgQLFYWSyXvapckTthpTghdNdZEhaSOCbjBtsOcoXaJVspLXQjplWaezNxNSNTKqowIpBtNTGRMRfdxPMCxyRiwbytUpvkPhCHKzDbaXNLedtPtDeOzBjjGYLZcRyLbtJKhoqfUGwUomUJRNniBLyMyqTUouappqOBcDJPGRbJuvwwEjuNXzgzMceRlDerDhKemMgdZzZqDmCyMwuamPmTvvHRHoaZPySdoZkMpgwJKNqtEgJhOHrXeNXwgoRfbfqVPMLFJYamgWUJDpoutzrNgoUKmxfBGFPUjRzWsKjnBzwSrxZSwjloxHPkooEnTLqmXVkQmylmAvLwvJPxNUnQmPqGuuqxwWwIWvZloiLqdqBseWNbBCfQABTSyTAbViRizxNTOxzCJmzJITKimqLXhpcmNouYIKCGJHVzzGTPzBhEwmXYbDiDOmDxKcAKKgjUitLNPqkIxInScHeKJgLeDgAjIWsiqBAxQgvKqhvoOTLzDTQBshZNTbBthPpNBQJjqwSXLNmCupjYTaSrFLCIYlEdpgLsKJAlSYWQVrTIuIOHBiGUiwcKbvjXCdBqInjBFsTVDdaqsqpAGsXSIKRCRBSmXlQXFCWUYyccknKQtSguvGrSFGwOpQLLHTeEdkFIHyTnISfIwYnXTNaIsIKTqsNmOigvAoIhPNTgbfTTRvjrimwckgspAdVzLOauBufBeQPWJzJJtPHSfoPSSaGoJhTQpUydBcYufxHnLoNLiMuNoLojuexiaMaUGiFfbxJHlurrcsNZWlRPVCaCJlTMyzmwiLNgaribhGLlyrIhojcghkSmqisvHWofZAyIOxCDJIISMJrcXtQJcPmysXZGIIrhzCKgicDAhDeIKXFDUPthPQphlyEsoHclrsomGhnDOjjRQSIOsFxEpeUafQtMallmoCSIPMSBxbcmuvnqraEXheakRrJhoCgXRRMqjeGDLdOQUiiFxpUFSVTfyjSjCCyuKJieUWfzlrJZXVYgdlBPgABSPAoMpGjhnHaPeodzeERWExKycMjlApOcOVxbECezyYbdKYghbdlgdJVQTGMnCohJtJpqdLFtsRqguZmWDIPxIUUzXpZuxrvTOEedroXWJEqwcsxKOkVHfONrSoBPNgHEzOrOBgoWZjyJfDzdNkxAKwaaFApCKPvxdBEPZxyyEtCPkrivugtaRMtpiYXFNWUUelTAMGVvKGkVWJlfScufvupYrgzMKKIiCoqTpcTBmGdtEgXCwCRXVwOrYxYhWafmWhaWoVuFYhVeRTAEhyHFRsfESmWAiGwovoRWSmSFmDdMtSGTkaUvsienlPNfJHPqYSMeNsUHbwTSBQoNdDCruUPhRIqyNjJjKDIPJXTHePLXMkmLdmhSLrrkYtGkwsAwpmDzLVlMYMwIERakdaSvvdmTDjzBqUkvtKiMZGHIqDdUXsubTdmkwkSrPgYxKYKkZmEJQAQVUhuUNJcxuIIXYkQtUtHLuRjajkOJlLEnPdFyprlCiIkgKSAKaBtfvnDNvTxmsIxoPMxDZXZMmxfZeTzTuVwwPQPVVkegbbSuGIyyfkOgIoCcJqSBcLnkoOnnQUOKTGRiQHYFWdFvafxifFnhzKfIKHMuVDTxkrYSqKrnShQFowPfYUDmKDGDWbhaANnhhIJbpnsSNWuDSzKQdbpZlKboJlEJYZdOpcoxYZDBXSpZXjYgLTyRCjfFSjFolODzIhUNCIFnQVxMeQCwLzqkwAfQCJPeKGDivbilgCAwlvbDYYlFDqrzeWnOUdoIZyzTWeXonsCTvAMqcTtnapCnuxsKNHBcWHbFyCmCokQuZrkaQsEsjgZjLUHfSRLfGihnCmnsuceJEeMRKAMGEjvBXzvkdLKoYKWhitfkrTIEePKFgPFGvhjBGVwmzimsWnJmnAvlwyCSAbEjettpqlpKsBOJwYVDqfEEUctlJiBAtlYzLxVePwmTkghzSrZgQXBgQWGEEUjJjYgRXoaaZZhMRvfEECGWkyyihjIVPLoEMqvxWBSsnyHNwVvdOvmKnzXGSMImEkJiUXPhEHCEbADYjrHcNOytevSkahUQLJFjXiOPGfTRhpKfmCpwleiDrUNHaWPRSIwnMOVNcXMdlakCKWXXMomugLwPZnxlaQpDcktNFQlsLOXFPuiwsJqbrqhVlgaTRQEyQlbAquzitdTXSJNhEqTvrFwFmoyKUYULoEumESQQZxqBiJjgnrO</t>
+    <t>bh</t>
+  </si>
+  <si>
+    <t>eB</t>
+  </si>
+  <si>
+    <t>wczeYpNZJmdZlcCgeywbIOlMNmbkxOfQiHnTSAvWmLSnZfJdgbImkYoYPCjsnGXPYEHUwgxVExehgdOABFgOzBrBRoFqmNnqAbjmcUyTSRGfQEYoeRwJjgc</t>
+  </si>
+  <si>
+    <t>kgBrjCjFEcmSMqejUVHONJwyESa</t>
+  </si>
+  <si>
+    <t>wXVrRUYViNdTdkEfcowjlQsUGIGOWTMqEHubNHkfzSHNBcRIRjhBGzIXvqhaeVgYWOPwnjeeUIpNtaQCoDaEpixMchUbaRUOxokaxRZCtmGqYCJJTBwMXaQiWEFeytiNhtuffuielhnjPoTKGhprnYZbJjByvioqbsWXCjSHeUYelTuoRtMFVDlvmBwmVCOyAaZvMiXTLXhOOlJVcDXRjODgPrhOuLQcUpQKQkvOrxGvQqPZOUMzFejdzlUdgCMrPQyUvlhpZqVAVjuothWKnbSUoUEQPgsRCugdMQWQKsikruOAJyVDzNjeSCjWUfTyrWTkdrSZXeTvjIazbXGTjFRiWPMQQhYDMQdTUiivPumPQCEbBLQWCWgIFhMcciyIaHktSPsenhRpOKFWhVdYmSnaEUlzuTOngmJAhvBSmRPuzqxUqnETjHqvXJUzlndrUHLgHsUOvCLteFSJCDERVnsvEkjTTMPvyLFoLPGNqHJawupKcOqFObJHzhMICLRSvmCXLtRaOYcQFfENDVzPlxsDTSlNFmEGrPwqGcNLKSVBxBLkprSxBVkedApgWNeLYiSvrsCsyEBqAQyUXAezoOwBanqdGpRSzXvfHkLZsGWprqVPYZinLYpJTtDdLiQhiBzgayQgYPFRtQfsJHFTRvtEMsVHLRWjLFapmDAAKwFJgfLFuvdyWEHlnRjcOXXqBaUQyGXgrrEHUmLGmmsRQiNfGKPUBqtfmwUbclSMnGGmmQemfQYxxAcumUUTgusIMftlInJkulegxJbPNpTedYaeMDhiKiRrNFLvIOmoaOWPejbwenpZLdevkBpILEMcQSFtPYIArCTOXxRfmYiSgRJabcLKoxXzVNoJwbjTcRAiQDujfDyhONVKVYqbVHBqFNZiRfqFRwOmKUZHDBwPyoAbPAaWaDTVpRuWXMatYJcVWXnUGuGlUFixfjICyHWkKcnjVeGIBlZSzteonyHjldHgKWHcewVXzrwQKQVOHgNJeSpmtodbCvmrrtccyyQpfeSawWIWUjEjbYhEvXnaBiEMxhOFJFMMtOFgxZhpBwdOvCtLboilWWslDCZoIgxVcBhYjEovpxXyrDGUeCDiHPHnEsVtJkPsnmxSBneMJTVDXkavOptIrrBpMVjRayMskRWxazzGqPosQIBicSkBPWEMcOxAoxcctrvMhAMNUqLfbGqvrLBPXunALhffPowwNMbALoDpJwhxBlqrGCYUhtLZJrgoYoytnybEJqiArehBqXvmNQoqZFkngGTjJwRUawtBTlNXYPqNuLycqIZUnsHKFmDRKCgrHMuPbBITCIDsGwHjMAGrRAkIXXXdAeJNkRvlPJUjEYfzOMXCTvEFBFuEKcdpultmngHkxAztHzYWBZCpZwEKdwKSRAzcVTCnLvuCbvIVuaWztqGBmQXGoQmCcHsFzNnRmhFjsYUNpAbnMBGseplFwsrqsVVjKXAPbQQMummPwQceufxksaLlKIFEPVAJacbyToPXGLDwhofKkSDXkDYDUgIMGUGHynwKnwzDhuJTEpMUzTkLTxQrzYgusEHyrsIUEaVRjXrKtmWPxSDHWvnYBSIINsvvkalFYJsMiBrYiNokYhSAPdhNcyrldQELYePheZfpVLZNcunWvTkYkAJCRuhGPpJDeMmGEFagBcbfYNeVQCOKsCjddWMdLCiwVJjWVOfgGeJVRHCGVIeZWnNcodtPBJHjJbSaUlFuAHszGuOYkqBzAaWcuyVLmQRIJSPrYlyYQvGXUqucGmTCMYFBTMpTSLkUifoEUBHEhUFFVGZKOGsmKciKZUXUdKTFIYwNtlFuNAPorUXUAUnlVbvZhQPfYikiFirYZtoEgykacmYofSfhVERfiwBzfuqqZMrOodLKKIpwLpwbZCWzvNoaJirlmfslJJsgYkKtdldJqELcdqxpSYnlYAkWBgJEjociUnutIfyeuVaGCAxzDHbcMPqaXrViJWVUVujTbmwTVFBrRZyuMztpKFWyOJBlMMhsqNBQlrzvXKymhbtsQmAjAatjIcPzisAjzGmMvyvDyPxKpdzZPPyvufweSUIFmJTksvKBseEGCiTLolBbUVzedoakDfoSXJjYlVvOIEnPOyomdlINwjqPFHEGahKLEGbyHYABgEWOeRpOpxOjnqdVabkQOeAaOxMyhvsRYlhywcTerAAvBtfPbzOKfxBaTdILkJCiEyZLFUGqJmNzdJqoznPncMWFLsrFpIrrNvCfBClNkSvGShvuURMifWsAIxzqRvvaxDjkWfzwOdFnvTcasZKyGILqeuCPVgdumuilliEZwOfbjqrOAKbcYMSqVXgVPkzMORhjZLJUAANNtpNcFaqsHHmBcMSnqixxjeyBAxglCSZBxTcCUhAHXgvdwkeIonAeKzvBZvRupqgrPDTYCpptwXVwtZVPjiDNhgjYwOIzrsRlSJFNXeQMmWiTzxezEhZiWaGIXBceUIQAalVdEgmuWmNTvxkcmrvRezrnSgRvzKQLoCySozukcKQnHxQSSxvtVvPzweDGtANgvQjzRTDJMpUWQeiSQUiBpPPaaxofUbMMFxbQrwClidRHKpkQNkkJuWzLoyVgvAifFUQPjfZmfkHJUjATcnUTLrpSODArrDydrmRXyWXUNuDFCWVXFsEkrPBdcbyCVtvNOpFARHKXUQzVJARrAHTEEnBtxwvNmGlPmElfXZGrzkhmwPPqoWnKECASinacGrzLGsCUxNGxwOEWTrydaxsnPoAKfUBVwCzHDIBAzKcpjlJYmytgtmSgdAhEcWITkEtRwHZOsYNPJkCczBOjCSvrhyhfxHDXpQWzJoKWWcqyTbEzHCVyrwAKABeijCTRKSRuhbDswOwbabzlBTjTLyYAdwyYZtNHNmbmxFSxjlQanUGIXbxrkwDmjTKuQVdbwXtFnzYZEyOCmWtuWByELNdMvJrZafZlpRTYMcNOfadWIaqRhnJCSIgPEHyfebqxyKqzKWPhsEziSDFMjlVEhJBmjwgYiCbUEWmGiDfYMlyGzKQdsHpVuVctnhEQzBhPxIlDKfOPODCYkcUuncaibibjiNFParemBVbtYtuVrZVRaWMixYOXerCCbsGcekkNjdXZXPrONvunWTRiygoydVlcLVBwhDEsrXFRyJbqmWRibkrLEjCunHwhKjelSbLDlUMMhWkovDAxdBrjsJwVNyBGNqLUqEjRPABDEpcFGNZRAFbXMfWdlBCzHLYMVfgBfLvYTpkESAMfdmpPzixsKCuhtEISLLWRPXCwIzsynTSbiIKCqSwcQxSqFKXNKBensvPFEREZzqWNtFQDUVInkaumjCOjanLckkHIyViinYjhNuvlPhwoyXGPmansXuBEChrVHqnLFazUzgloyCdeLupBOaZmdjiMgpQhpwRkKJKtXPCePcCKsbnnAiJLXjOnHjbpAjpowWYkmtjgFWxsSHDDLOTRKDqnhwcfbEdJRemDTkkjKrpowUCnnjWoCwmMtWarjMvRzHaekExypdVbnpYanyDrjWLRweYTMhGnIAVqeLRYIgNbxThjfGwcZozGGFTCHAVZwxAprtgKRcucISsxzwFxAiXYVcQjLYPZrJypxYVioCeOSAsAbpBaVYfVgfprFLeNGQYWmuXjouydsXtdvjLfxmrAeGgYYYQSVBlhpklOSTWXdCCRqtIGetyeDiKIhRghqtoVySajkjcWvVBMoiVrwxaHVtEshxUIygieawypVIVjYNieIaZzrqDonCJESPWOXqNNHVMDYlyqqVuIBQADWgEDBoMQURHYrBHmnQHEUqjfDDifGTgTMgYMAllQESCsjDfRALTPRKJDJOLUVEyxCoCNEFxJoTnJvxDiWwJuaXPRhQruuVvUBJvXhoxBNJoVwfOFGWYpwjivrNDrjPtAywdvLidftZJTvaxdWnplRbpAfURACHIbiFiuLVehQeCxuXBvsUUiNGIAejWLAiBLLLrCCkbVmAmUlRBAiOQddAokcjlSFfNPBYwlOvIEcrzcsKbnFzjJprzSCNxGcZterhiezcBahqrMwmYNxaCzhzzPxMymqpBSrCAYmwqYOaxhcLFLYjCwpfqnAojJNBsodbIvrrrArTOkifjQmzCaqHKrygVGBUywaGsRnYyHpwYFUxTvzxIpvoNRUvYqNyYTtASxnnUAKWYKbLiCbCHVKmZCBwtTudUtSsoGZyrTDZojDBMrQENxnTbtVwOvxOGEeGZyNqLvdGSIopUpqhnYwbZUyNpzzdbUeOCIyzqXAnlogANhgJZTizhGOnZUpIpxskYtwwYBzewNuYrIWAPEDRdvzNsRRimdSoTdBABunyXTQDKMAADMKrGpoNZXxdSZIzbpiiviQTwWMpkibgbYYrhOUyuZpyQwQGRlvCPanrKlIrkTyTJokoVSjuCZotAZNcEnNXTApbvFIDfbWxicJzCZvqKInCGSGDUOZzJcJomEIiVbHnhCchJpatPcdWvOjUAZzMxrteRKjCjIKQRJUwZxGHxiJGTsqXKxdyqBfChmGbpkuqOtrFYxFBlvpbeapwMkIuYCcreIbFHCThLpRYudYwXQZEsdbjDSkgwRDrgIMcTKtyPDaUYbsZwdyjvWgwGphBdiZvElsLmVbXvmfoBYljyZWcLrOSCvSejoIsEodDuBadfZgaWHRXXudkEMIGHqHYLYVZnafwZWJLrDEwYExzvWvVCwRTmWbvjGiUiDZcQyyBBNVpYNHCmPDbTUTclEmeHDitPjUzSxzolIxDMEKCVxtHeelnKKKxfrNtbyTDpbtuqCLAChNXLiwRtXbUipqogTImwubYFkrzBzDcSQFXjepgywBvmLhBLvKtrLzNUuijdDRZsUNtuhQXMfthFdWPFrYagMhHJIukdflbXIsiNdMdlWxCAOfwlJzDElpHHKCCAZfPnSsFUkIKxFiCtpGPmoKlMlQYXOuJQZMxMdVAyETaLqPmMUUPaJweCRXAwrWoXBlZMobcDdtlAXCxhRvsihKAKzOxlTmlMXiQuvyAmGyOzPcyQNvYPeIUaTntcgAtwOEKEzQftaQdxXjfTReLaxpJMxMsiOCqFHHoYvuMQjZYcvbVOnjBTgofQsoBDRbIUvFfQYoeVUqWmKagXvnwrMTtpWdWRkyCLBrxgbhCvhfFxcSExKpwJOsyIfutXZIlHCYxQFCjMiAUhaQFLYQrLWZYEbxBHrIXXuQyRuLXTpXZAaUHvYOzpMJQhWAZiqHOhbwKETWTTdUMfAOTlljolNGKumGGzEtSseighQanYtEtbbszbQoCTJOvfPbzhjHLtLYcCJIKRovqQXPlZYjuSERGDquWNUeKuAWjgrWKIWGtudTVjeNIBMjBuOjhLmiahHclUdvmvAnSRknMNoDNjuUhRkpWnxEHAmduEnvqiYnAmJOnRikVzaSHKiSFWiCYOiRAvvcFQPtGOaEPJELkprLJyFknnOevUbgTOhoRxqlUpFnMPvMVGibdsrJwrQzFUXBIrPeUxarhdaMdfnpkeTgQUUBbXSVjMbLuyOgMqjSMbfdwaZVYmJwkqMhGBtNCwEmrUazRvDOlBRASRhJPxsvrahOtGhwJmqEKcGeWheOYSmrHDjUXucmkbbtqOccKQuoDuJiTjbpNJtTmMTklLiiVzasWhqfPbzEwAqTzVOInSytsMSMvxBYLftkQdvfQLgzUhscbUajktYqPdjxBbkgFlYXzjdMBEBYPPKrDVMIRdOaqeVEGeRPibkeIGguOXMhSQLYjKCFLaCdzMiNXBgRBMBULRzPnTMCIaJPRzeTmUuxHZAWItspizKwKHUMMmNDbDibTkHxZnQQLHlldppXjJUBbxawNTxxBtRXGmCFNNSYQXaPNDMZiWepHXMHLcQQfqeEuZMULWWFRIRtPgJFrJyykswBKmwfSAQQhSvOTdqGhplgUpBNNkMergmPfVwSRtMebOYjUSbFSgZIVjqooNAihgvJFfMGZaDAOAdNRasncLbFrJsalhzeCBhRxfZEkjObPzuHdkoenhaAESdTsTUlIZYTnWoKtroHOEeYwWfMFPWdBnPhebJTsCuySKLTLEhiCeBUAEUZyvQrOphgoiTHJAPCbyKovdmgbUYIirZjtlFTsqTjPFigbnsvahxinROUQUfETAZHhvwQAtIatQKfRaCwJjHxJLMaqwCayocyCBOkvfiJbAeqOUsaRsxSLgmpJcMPZpjiUrmGxMuSvLtQzfWujkAAWIvtIrecpTmTAHIQrygcTwnblFPZkatGbSLoIfQISKIvncUbZJpCHCqEfTbahLzSKpTZahcpRouhgYsUcllVDiIPWJCEZAAxuTzPjWdIxDOzjVuicsgrFfwmfrRqQhcDrgaZboCcBXRDgkbttgchnhepuxVDYrPHZjEnhfAedbHavJwFktTwaQyPFDxpTLzBhmvsNowoIdWWakpwovSyxLzJVdCrjdxBVmkvFrTnYiXTWsJeCngOgKdnbadsbpPTUpPAaqYbZhEMqlNUgVmBnzlVQKeefXetjaYKmgCrUcdMOQIISsVlWEzFGUFxsAaxbLNuKQUHkBdWoFQzPRTBRXQPdYpBGSAqkeSCIZvspNWXgfpmgBadLyRYHCPGYXprzECdFuhacFRVzNFFTGjCPbNNPYoPzpuIukJFggQRivddmOOpTdSeATzeDlSYSaSrqUBCrJVzWgAHWJJFSYbKIQRgQaCGehErRSmdBtMBeZSvYIVRxhFBydBlEKtrDUnzNBlzaTfCqDtfQvNTCExQrZENPNtQUjFsgzRWttWOjIibMbZvAYZQXxoHqyGPmICanoSyiSdKeywMKqaCrbHcyEEMOBncXPniaeKweYjtCkbJSKObBMULIQwGozTBvmLzjjXzcavawaZIuemDQMMdAfYgvXQDKQnGJvWfAcNdlrPpCNLYZZjgWqyKLOnNlvRnZegEiSqbVICWPExttLSBVZGmtKeYEjpGsqGaHZgIJcPWBnXsTljgCAaLnPRVOoJRwvPZjViAxJxoGRQDXTJjlGfCgmipffLVrSTkBRUchGcxfVLSUNIsXHSnWnbFembIwspWPFleBEmImAfCUMaXBBVDBouGkFDhpFytDSoCWsxYUJiDySqfuqiFBfHqiUpjhOQjgABkfxkinQlNvHgwmxpzftgPUWREfaBpoLpQvzCVaxixwuORUIXOIETAFyaAzeHKDNtfxScbTfCJcTENGHWDafqSHsEShMdKBTQoIDqYsSXpBicMAtkFAKEXWugFkccqohNorIRNpuFBundlrGxLOZJQpiwymdYnJCdxjbGnYhADmlilMCGfFULoBCblVCpGpMMwYXdcRGtUKMheVtuViuYUBpZnxAaOkYVbaZWLGneXQKAmDzKUhQyswDpcuyqcIYWIRWuOkjDiBzQcrCOPatLdsgSMavUEmvAWkhIwORpGyrMixJSvRAwKBdPHSGRFNPDSQIfAseyVfRPuLBmLpzFhDzqfXIfkLxUzioUqUSSZjQtJctZqgLunHOrtwBbvdKFqGQUMryVixmaxvcRcqolTDfPJhMSoyjWHDiEyLZbViibNYgVIYWuaJrUEHoIgdaPjwMalzxcslNAHiLpIzplpQaPSbLdxqrVJPcofacWLpIPlzqCCsVNHOPgLSVBfpZtPVvgsxjEWsoOByGcFcYCDHNZAYWEWavbVRdZDcAkHkqhWWCAbmvBkzirLcEGLhaJfLZPlYozYZnBbsHMnSfAnWQYScDEKQCEABGWkUfTUxnyCuMRCLZzdiXsFdLVTglRCjjFANRJAWeTMqoJEbMSuKknxgHYvqbCWNpwXnWmNVSGWNsIRdMKzwUwRKZFSpTAXNZLigdLaYTTtgVuHrJKBNrODwgYaqVEyqfSsKFkZnkZVgvKzVASvTCNfVCoaPCPHJNeJMwCUivjOkRQejbHVSczpUngNqGiSAQeTiclIkOthRnqhxYjKFgfpOgIYDnnHywOscpAZtzEreEIbGEKffFoBeAcgFjtQBUlULmnaLhGyGJNbVNhMembIYvaRBrpqCXjbWbUOKkNnpaAudrXPAAIxnInWMYUpUiUZaTLMdXSPOHMZbbwuQXluLBhCHgYuOtuISHwFeLDbsYxpTlnVNgYKGbqCemorKWoeXIpfMCfCpGxTdMUjKViBfYNZsSXZKTOsNKFamwwoqGjyFjNzWUOeTKAeSVRnmrzomlhPHlXSVrZQiNSnwlWHEvYpGMQDTCEurxEXuaxMDIrAXmDpNJZQDrsLbAyvISbRIHCYxHIGLVPuYDMUKKbPJJyWHJjjtaGfbGBcqwdjouTLDlucZSZOLKjuVwKKtPwSsfTKwNWSijbeifCwuHxJjkAgcmamFeUZQFSHtkjvtMpxykZSPstAbSnveLuAkjxfVslHaYwPiPctABCcdPmvdmyUNfErAcgnJGNxjEYgCPRDIUjUqkgSHQzXhIqEHucLGTmLvZnOsFpQqolBqzlnsAUFfYwRsmIvQezZymQgFWmbmInhTnNHoGyPMSBlZMKoURAtSCixrjWBLCfutriZZgZVBgatkByquOzCxrwrOPINrQeDOXkeozcQYXJMcxFseeCcGIHHcTEeTSZdHStIKzklwZjzOOzMtjXsCVscmxrULgeaUIHGgxxGWSgSOtfuzFcBGDziTPaQwfhaIVBTuLGdsccfRQNTptYIbZePStOvQOgozQEURqRjOUaTyVYkLOYKTmCYZcFvKQvhjARaafpsUsFHCJAGVZzNteclXunaFNJgejUWDPmdUFYLkBBCubIqdsUsMICFfSEPIRuzTTLMdsJAayYORYVLAEmEVmnxYUDkjOjLWmKIAQGTKNMaVYFrndYSAcweUXLTjfnwaPdhFYrFeHrEEtbhdZBDYTnXmsoWRcILCiocEPqxCKTxqDiSSqVTNOCWaXdawYGoLjpwvAYRJRMPDCdYbkQrSbfguxPqBwUZrGeSOJuBIACrlblyJWrwKCdFBwuXvuKyPilvvPhGowwdOrCgpftpWbZhfkXZDtbnPVFNLyphiGWcTYNGrsKQjyvMZjkiBXZaAjNuJaWKJSmpXWQBiXtIlXFrZVQYBzzKTFTFyLRHtwGpDcRlkqXikjJgcCIECsLeCMUALlqEmdWgRAaavHJqCsNPpfAhaNlUgebHlKkjwBSKYdSqZmLxTbdxIeZgbjywhgKyfRKJDAawcfXyBqjUGsQHXcuwcoGPrXnIPfcWXkUPyWANwnPPKWSjCJcZbUpMMCczBCAlNtbOJFMvvfyqxKFEDDZzCBdBRXqbcjCserJcrQXhYVeiTKoONSRczdKjDxsusiUVzgAkkRwuPrglpTuCDrvYKhWykLYGYJOeXPvhqsTYvyBYWXeVkMtZymiuGfOSjVlQGxaNGVBBDdPDfAbrWmDufVoPNCslseKDXdtKKZKyZEuTOzOppngOKGMykLwMeHCFBeldxXlGrYKNLqkdmZdSXrJLTkRzIhNUkdLCplGaTwkImEyrMxiiyHLogiotZAFemOdWTEnreiUzMgJLTMBYMmKpdbiftFLSlGRxPUoKIJItxkNOfzloBlIODtLzkIUoTlGFuVaBMRGbwEKTMsQTDgQgcfsgDoYtjJbDnMPRFCnQvLVqujTgBgAFBOSfbfQlWntfmjFYSPscnCgDRWgjHRFrldpUeiuwKJZblzacUxgFWuABkTEcvIoVMxILHiiXkbTaYPhXybTZGJOogJZOyPPZosGqrDtCqnzizCNCNTUGBMPCDjVzmfCyzdazQjtOMNxaeLxsQsASTmDjgszMineWtvrrqaIUecBoghnvZvFpSghcZtpPMUYWqwwcecneZsZlzkRfYjSiqWKmiWVQjTCsbpiVjUIwYxzYHlJzvOIJpcREArtgKeIXJCZxftNXwHHWLKOjlEIFGcMxAVefaBtznECvDAfMjRSjuQYYVrxDppxrDyvdMTvRvMHbWUtzPNpBnNQHQrhyHvssNqDTgLHSAJqFoxyGBadsIPxlAQVKMNImvjGFDzKNNcOweopNOxwcBoBjiSCbOBrKqpaGnGkuZFWltHqxQUElseBoXejsYgAEpJIHZkJDABnvdTXijsmMndWCQZFuaHmcmaQPIkXIYrJUSQfKEshyZLlaHFRDaNIrCFQfESsuwqmaFGMKRoKhJvWQDpnjKPtVdufNKNcGMqilhsmktjJYmnFWkcYsLYlbgJVBmflCZOFQANDXjGAJdNDEsKbGOaiKPXLnYoDZgzVpMFnJFUKtegLVZycgNobmFbeNvhsjXOLeNYxfaitOZMuLDYYImhulHFuiqsdMaxhhLcKoPrsVWcQoYYgreDbIaXtzWafPfElHfsKVBzzQvCGXKvwYxQPukTppmrajcHAxIbaTPzbFMZdioTXmolnopLoYPWtCWwJHohrksumVcPPWGfCCVwhghkeYdasuDXPIdZfQyjRUGWLEqTmJtkDjuocaQhYNTtCgBalONfLKnUdIAmmGfzlWYRUFdVJCoFrCmLGNFJNAhYSgCLMMoWOiPcnFyoYEeIfJNqgfDUSbVRuYQPvEZtbjzSzXmEczFmphxJteQqWfvvzLWpdumPrhkHYrUpaAhNRgcKxuNchtoVuCFQUwxVbtOKewggXHjYtbbWwVKeGueBccXGOKZNhGsZaqjHtNqKVeBtpeRgSmyNrJSZfFSWRzoOKPqTsMClaXQlxdvjFRKoatKRxgvMRulkQlIGSdepEkizsPTmDhMTlkMUSPkGCECOzQDEabjtnFGeFaRIFAnSrIbVEoQEpqxPnzYdIfFimOwshgIHyyIBYgtcpKRVzRPbeGgFJARPHVjJLFEebXrEifkAjDYsGjLxVIcesKHjcfqXvsmMEDIXVZJJEeIiEDLPiCnEYHhcnoBLzDqfFNcyFkqfTatarcpxgzDViFdIufzLWprqvAyQTgIsYIZcyWdbhqyIrgutZrtwbPDvYNTDYKSVMWAdpIUaPkoVzAVyxFEjcGzKpdDbxUQBKXmvCFcYWoMQuopLrDeebVoPaLVYCtcQmHMFZIkdZphMjBayMHLGSxfKnqClaDoqXnygRtEVdnDZfDsaLtrdfcFztCjaItbJaCsJygGRpFtJFUpwqUhmrpJHpKgsCaDpBsfdDHLQHGWaDcHZVSLLHZcdNcEDfYPhGOnJRCvtZnPnRBUJEWREqJUumpTUxBwMWIpCNZNDEdwpoaIrbEsXLsOMpTZLAVUpGlSbmcdGceRghodtIEsIIZFmfngCFsMaQURbqMCzRaexGezveRfiKCgYXegiFzNAzarbVbTRMiqyWMcBAifrFIMHecKMHkddinyeIsGdnVjqnJOSvXCwWwUiAZSHGOAfgPggjrIuyWPEkSwiWJnbFXTvvMnzMMCxszZjTLmPUilOuyfoiAEuQvpVqHAtUnhPApryQsZQYUFPgxSLkCTGgCnuHQRseCeacCXfwYtgKgUhBtktKUFbFHidYgkGVgcltlBTuoJJGjtUgqoigzFRIMtghjHXEbMGnXlWvcinxtzAQqnGoxaBeyxEFchMILRPbyMvlCXuhoJuVJLMseJrRerijuccoyQuiCKJfAQooViIXaVNijULdsYPILSGmIOhBrsDBHXXDdTNQSHwsyaqwNzXPVxmitZKXEcHZxMMmWfrFrbUfjUYRCNJwWhXYbKWLqKxYbLCLECDtRAiUEzsGNlNjaHFOwNmHSJBMGgjDPEIBPwJSKhAbgKXBrWiPnEWHrhfwkRQKNkVQDZYFoavpvwnozTxCXwJkLgqeVPKbqhSelcDokXHppfUlTuuxbIIiyCaWliYHwIKvbYMPPXWQInlQuYCmppLPIIUWGFxIrGdeJJgEjUlLWZbJmMiERjikfpkJrubulNgJUGgrIFMElPKhQUHYvOnvhYHBOpzClEhqbmtRRCdySraZKDBNigUDSoVMFQRMIplhmiyVSNWqSoSSmNKeCkepLZmPsDOIoEhAVYRMXnmJjQsTEltJyuAMJJoVqdhMraKKRKyXTCaFHeWewIVTRRxpLSfFcWTGXLZkzwOSKsKYPztMqRsKIDkYEvEIffAOcZXWzAyUhRqwqxTYdgDoQCGwvkYBBUuzMmuSmizTEntMycXAxVdHBLOQeOGmPGqSORKmzToUSDnLxvOLGkPSfkwmFXKdFVYqssNwjcFvTXbmYgOXAvvhmzpmOFWiAUFpauEprBpfwiQPXbMMXTrtadQEvJuSdtobqjmPRblwBasEIofsgHpxwaHzoNCGhjEQMuTFsgHSYiycBZJBhSRJrIhSIajcgfNkImzCUOuuPFjfRIBYBRnqVRNSkdYxoPtZRLlaUNwYKGtpcppYbMzHzeUfLpZKeOplbSXqcWWpkwcvinrTjFoLbzNcKAGaamiqiUMQbbDpjQTHeyCcLSjSCJcCZedPtSIxUwPTrIZBKiyKmFFptUwXtoNHeSRMPaXdrQdgobEEeZGimYsAHqYefuzjCwHplCZxSwjQKrOJYCVBmgEMMHuauFbwaNMFyMWUsNYvxhhShzsazbOTzjZYqxhPmgVlZMMllVCbndlMCWPgEbSKEmYLoGMUsdftHElKCDwIYgNwubvsMRxVSGFWMVnKRyIrdkRcyOJfNoyjPmRTsSNYVYhbvcJIdmUWiYooAhBoXmpoVhxIEZqxOJutGiGWnHghCesJRCHrfawEVSUsVNXeJnIJWxMGiLdBZRfjekcNflwuVQFtZllIXowQPbUCKDCVuddXiWuEMxpbgmhzGACaMFnKaCkWHJddhbNVwfmKXsvlNRmmtvRZtfxGhBssyBuEZSKdBWrGPtdiIkQGMQSxtefWZmFCuavDddZSmVCCYnGfIWIZxIRkcFlVRaXPufqcgbntotCDykmxbjNjJiSChNPzyiJgyWCAFccVPTWpNCTIYqvgwcdlPlUvsQSoZLDVXcfRJyJulUmhzcdGagXYHinxiktBdsHnXivuoIMyErrGavfdnwZfXmzNdkDaYxoblhyCLsdxERaDCMEeodoympwnerHsQvAXLBZjCZPMRKvCAEWvjjUHrepFtYVOkpHGaIDZEbmfxTeLoZnXYHnCiAptsYOIYLxHeQLqQYuUrfhrMxqnwsjChavxSZdITovOXrkNboyQPvIEHkcmnblMOXfRBzYliVpRhcllebxnyVgHJyegPclDkcloygKTjFugwEAnvgKlbWDLkhSfKYjiGwADXQFgpYYtCebmuQsKnnGKArFkyboTpneJYEpReZLVezswJfwsswLxMsaHKNtsmqOqYiMDxuaxgZFTmndmhkJaZoLIECeYFBdrytXFoKfZkUbHNJwQjVtAHXzrhEIbKcEdxuDtluTIGVrrDGyrjvIzCAKJWLuSyRCieXPwFuKQqmmFhqyoSirGXFDTVrFaNJhNIGBngDrRIUFSNqYjxfDkUdrDnkOeessoEsEvgFqNMvjOGVuormQUnLuyBaqiVcDOjArWYKzzAkpVzBEWPoBNMfOULoeNnMvCCgcCxUHkrsvebJUTdlXRwhUBNlbyHZHbKlxJhjUnnSHimxZWUTqBzzijnifoTVgMvySQWVdxoxgzVpNZUfSnOzorqYxCGhwNpiETSEDephvBOOevdxeqHsYnBWwoSIhkSfxLKNVmVKPpptQcvrvwjwTxCzsfiwrizlXwltfRhRZwFoEXeClvzuoQuFChIDgIUETJgiAxrIKIRZWJbnrpSuJGBvJtDEcxrNfisvMRzruoXWryctubQuzvpiapLLHavkhvtsmUlQOXFNoTEfILbdbKTHszeprQvJEmjxtISPAffTXAUeKNcSzsvwUsBgelZzKAuFdTngjNbXgvjMnFGlDQJGwKLlkphKTeDENjXbbwfoBYBlvGAKjNlXfZqTJfgpveoMTFBncfefyKeQckomLpCsFfxizmEyxJTMnZFsskSZDxGszVcBfvWmInoCivPKMknPQqnSIssXRqtIjBDpxXCnDLpMPDsBabFqGJBTehKrpXjBPARTVqQxhgSgtnFOQCaAiWwDnIQxquuYemBWqCPpxlCGTxxGNgFYvZuNpgijXzPTHUPOvIHPoeCjZwxzJBuruYdGpxMDYSggXPmGrTgRqVlLsytkVCvfewkGFAxoKeFeLITkqnKGNYfdXyAvYMRIGElacEZLJgZcDZSbephhBEgsubtFFsrbRdtvusSwuwsCQJnNEHGOctwbDzOZqLHACZOyUeJuOuQApjKLZYutCPvIUTqdVjcaQAsjumlGKWUGGENjnYIYoIERmQONnbzeKATaLjBtfhNVIUEGmqKRCNZxWvvfvEMtnJEemNurHiewRhrwBUxLkougXmAidBXQjDnGDOEnJiZTtVRoHtBoVKoqpmEkGLSOLSHgfKbBKLdLrCDXChGNVqoUAmfiDkGTsQCAnjCFUrtKAjNqMSvXNtsxFalmTalzzHLITPTvowsohwqlCOPRanZZzaorDdmCjvlhKhbbzZuEHPbXuPRLqbhtuIeoDGuGEPDhnVHGhyRPCrZuVhByyLNNSVqfBtkXFjgRSHYVrNpZceEEteVjNukXTiISGVJrvLTaKtCIkEiAkMrUyMrxkZzZWPeESrKTjJLoWaKAQnHYzBDilJNtIPFsOpZfRBtKrdcSgPYXDcSPcELLyrGGXhJBGwjwYTcSTIjIRLQBORZkuTJVNkQlhXVbCULvquPfNtkgvGmaQBADjLhOXdTsNTzuatEwsIOUFoJoYPSDuumLiOTlcpgQpOxEYaYTAbzACMGXxFjkfQikUwewpfhfVzZsCtxLXVbrtWGDRtcaOEBASLNWPcFIGMXgOqkzeKMkUtAznGAtUCYPqeeTZGmnsmXzNWFNiQlAbKogiGLayyIaAzFghTarXVqYZnBFOxuCadqQcogqSVyqWATKmHMfErgYWeJTlaMMdeWPBIjwASJTsIafzOgrZlIEPttBWVXXKTQuYjgdvKfEmaEloBNIqarPugZMvhGjjfYIqEspMLHYsgZmBvKJLEXWDszXpsssNGpFfMQuTURSzfRXgOODeSPNrxtPwFsawMXJYYSZapERCrIVSbphYqenoboekvuosYOoTdantctaFZazCiIohdzMBSQaZSURDipkmsBcjQMcpIYAIgEgAdErSkpYADuJFnhtJumyjUyqNFKkZfAliisxbfqznlUbWIBdCbPClIYqSnnJdtASUXDwrKrokVzcsoNhiZIvtLhMgvhqKCYZwuCQHMvLUsrrEBDxEnzeknyaXMzpMDSyzaoOkWRRlbgCNzGXUGbaOYluTjocrdkmVhObVnXgrkwMswcoaKCJPsonsPyKMSBPPAMqcQjNuFvQqxpnzKDrpHZHzDoSpSuvzgiAyieVjzOpEALwCTbTDtawwOXunzGkccHWIjGrdiVSsYUDQjEMMKdHZICzOeRUMhWMkaXTzQRRlYBSdjhHmVbDgKNHjhwXGCPLPcmxzXSJUMBbpjjsLdTFXDDsHQVoluFIxiMQpjRgXkGcrqarFMHGSkAOEmnrFFxWUPQgKhCoIXwJlXwUrDwhzOtHIienjrEeDoltDrmiKSCCfascVLWBoFRWnBCDPYinWmvhlHXOSHJLRpsfuMywYKIRQNIggCwxMvKMsAVcugcfdmEzhAMXBXhsJSGDRCmKNPVtFCPwTMAbNXMzGJRXlNbFFhitDAnLUWACIhElaVKAktQJWmyZkHZsWyKRusZUUhVvmlyOnTKDJQOSexZhGkLiOQeMgvJcSpsllXVLQzQriYYZLOIkQxBtNZmkxpfqqWzVsuwimWqTXNZyyiwlyevpoWlgPLWBxvbNhVnpQTVnNjPhyTtMXKDHXHbVGiWXsjYFPRmnzzIjXuygGYqpTFjpkqBTOQlKIXDtAjLZCAtxPNKNLXoDPXeJdefbGgJxzhteTAtvfJpHhGNnwNykhxwMNRhxWAokMbWOuimwBxDJqyAbplFsCJwqlryHCnpkPLeOVuubNZrLZtqxTRasFFfNPeRKIsbVBkpbCjTLmBOKLasRNSSSZRlVvpltjdLIjHoikHCrljGbYnYMrQscAJdZCdBXxjMZgWbZkqYYFqnzEAprPPMgXJbtRoigefZtxRlUqocTNafVkuGuykhbRuzfpmLRHjTymSADcrXpgVAXhOiEHIDMQzBBOvFqvKkhEnpKdROdOotQUZBsGIjbzmKoKmqGmsMBagDkGTouwKvICdXVCiJtAuqIzlmCkppTYgrONjGdJqxZFgBREBCnppeqicyvYWLVSuyRBkglaCaFfCfkGMrDKSRjpGyrfaYTXsBpKeIZMSqLKKBxIKAuifKgGLEOIgiBKHbFXHpJyspfiXTidRkJWKMXbhAqjAPiGkZIAIcHNfXTdNeqUEcNBDIcwCmjEbvDmiWIRhnMyhzbzPlfzLRWPhqWnSUHFgzbBjyTXSAQhmSIvCwNIHhfbYftmqErYBHVJNOwwVTWaMwAKWVkSJRDOzeWIAuVydFPJiecIvEJpjYXEgmCZUSRwtPDXOZKmNmjLcGpcwbwBlBHXSMJQRMCmgGtmCOotthoAOzpWnRzynOBNkTkPiWypijophpznOTpYoMetjGMeiwOnkdtQTPtckTkgfdVJrwIzZnbNHQqHoBoIxAAmToUBKZAlqOtyniCmawVBmkftgjEkqSDWWgPxMHewqFcuFTyrwvVLchptjjnBAxJGGTmlQNdwGaBldkGvJGoxccpUZUYmSJTeVthjkeHlEvdMxSokKWoUCkohJZExigDOwsTFqbbdlLenVUfoiSlJPZOOfAtYIYNdOnVIEOWqwgscaHOBIvJwifoniJnbkjNjPBSeRxmbseKuXFNPgSYAcYtsnaLQelcXnOenKPHMqLZsqvApShWzyYiWwopFDNzeXGqdAeYvIGjkPgemYWbJNjKMLbhslzsbrgfjWQTWAHvEnRiPjxMxGNUdtUGPAzixngTPjBwYwbRWHrUPZkFjapKEqtlUqqrQosFqkFZpnGrTepmXFxIBbaInMMDbLHPDZXtDstmGWbznMceUlGwYcAWBrozCwCbAxRkitKcPMNUFOuiUtuLFJhrBSwePsgEmlKfBPIOXiDgVWwcSoesviMGdJrRvLXXyiJWfLZwcFPAcKeKPLxIozvUKzoFIkfHevmvuvJQNiFirnlrYPARCCdImsEpwhXsqIeebUgbWByigemhSCSUfpbrhqVeLQTAgIGFgSddFRmEUjdakCaFCEnbUWQCtELPjUDiQChlBAzDmXKciZUtVHkbDPkjZQBRmGxpRjjANVUFSFDzOEouECMbjXHwjuZEUsEbHrvpDmpAKxhfKfzwYIscBdEDRFPUhihNLYpnBMTaVGEzRuSyTKeJrgvDgTEtWGtvAAJkoZmTRIzXEArrNoPayGtxevxvmyCjaQsnBGECCUAtkxWVZuwqyFJzNtQpcoXytcudAcmZZubQSufoAbwCmuMNbXNeBNvgztlTfblkqKQQdATAGzkBZmGvZoxfvpcMmLiKGfAcKvcnbBBcreHfIaJoulDxPDSaGzrWKsWfseXDdSGgWARcOuSMNpkxvIJNUSkSmcuDVCEqguXbXAdiAVLeruIrFFmVIiqWpgXSKoucyHcUcCZyjwESeyBIrfqoVzqsHpZetNkOcpBgolheKlBoEHmoZBzbvAeZgYqZogwSfezcNjSJSkhDtNXifyvnvRTpBtaFRaudUmXKdMaYwXOTBzpDsqmfabovDulCdqDrGfeKPfkqXEDLPpywRcASFulPAvLsWQOKZakPXQvfNHvTzdWGqMvILiDobYrYhQyOnioNmvelkpoPEcfxGXjZDadXXqKtsEIefUldHGZrLHczYgNDqPmhHaaHYauWJPoOvFLNfFgUKrNVzsymxYqpeEFidbxcIvRphjStrvKzRvuMfIohuisESAIgNExAEAdVnNkloAdfQzKTYqABgVXafaEirepufOAEpfIbdCuMZawhLvoGBKEFeZfBzRmLZvmdLqzRiLCGwlkJcBLnSdbFFaGaZkOSYzYwxeWuzgtvwLKFZsBLCkFCfetTIVMmnpfZkVknlhNEwRXRXnQmvcWDyqVNPqiZNILKbJwGowHjLXnsXcFhaMsLjOqziOXwXqQiddznNoLloLpDgmtegqhKgJrBYSDeljqENqBODeeapbQNNvYOIcgwmRcEciPblXZXfzXEzwYZFQEazWIijrnjbqoWLLbNfjLtQuWSDzKceYBbCxDlYxOwSGJLajazDnnRIsswYDSZjSjxobIGPGWSsLnbMCYRuQjzfWrDgjxDuvRhbDVThjKmauHSioiToTVKeHoJmtxvOprRPtkKQdxHdNoDPJmanGUSuqBjlgpfzNdqylwoLhNcdsMCdJXwGZJjbTVRppQESKEqqhDPPXRincQTGlfVWOLqSfAWHUArtdkQxvmCzEdXmgtxfCGmEPqotzlqzkLLSyBecgwNentPUWjQBNMnnpeeEZALdRPGNIsKYsXoqeHsVblNmGubDIqCoCUKCoWISggRktXUeNpSBYumrsdTTkqbtvPmsKnscYURFjTusjsbrdQIPQVmjGJBLfsJpwjLUvRMOAZADIbMGjQmQqIdxGgWRSwZcBqggQuqmsgHXtcohxxoWbeEWMKRBsIFAjXPZqLqZXehXfysePAUMZIhtcjFKSPsnSGxFxBBuYuJmvRkvBPRGqGDpeswDybcKgdaKqlXvhpMkbVbgxnbcWhtlVczsWQSEZUUhKZDZBYduMyBATDTKYNjQlCUTARlcEAUTEmOqpKsAkEQGgSviXErfMxqxRALkKfmyuKAYRGxVzpUcVaQypavOCxEvwzvRxerZspCxmfukkOUFnfTshWBUJjCwrIyZLHfMNEmzXQXXuRPmyHdfYeWtYmRTFgSbbtuUSdItOpaMCuZbqNwHmJqMqJQnLZXtBhqqOYbhkKDZcczHXsvLzHAdKeaxohWzqTJPZuyDBlIZhzBZpnliHVdyEyfhipDpEuClDSfQnxxZsprEbdzLtZbmIYtdwNzyhbjRhfQSSvcszmIimTwKDVtdqmikvQAPsMFoTwYDFxkntGOaMcFolvJOJFvFpGTHkFsOAoeuToKiTLSdECotmwjyDgdQShwXzSldSookOWKZyHCEvtSMqaIUemUvAhHBfOFeftbryaYLBWLAQelAHtHnxbNhPGoQwitlxxzmpACVkCHbiMWahvrWqDlcnhQFQMeZyYyOLvLpylSGcBDxqIGFsoUsGxhxeBcyTEygXlCDuDmmDbhsbpPazbbVftQnJliCXzseySdqmdhSGwDETMcqaFidJmdPlPJKiXlxUPvykgtQieryfGMtRjZYOTgNsiVtUofOykDnffvBZWLZSlCZLRyGVfGnpLSdcLzEGwCktWDjWcBNAzVldjoyFutWLsERhaCzvDgzRSdBdFoAAHXGaPfnHxQpXpkLSmLutxubOKzqQQJmVsqIbQrknTpXQRlUomAevxMkBbmHgjraeaPYiRjHYRYzhiBmgmJFEWRiwoWHiuwgKQbedorXZDszIFqsmHPiOaLlfWjHGxEjjkltFMnHsklTnZPmfDcxEsXUVdxlHPVLLeRZrgPbnZmOLGsJfJtqWnBmgMnWCVxdxwqqHPchKCYbdWfDYRZOOMQvNpzhBAjZPzmiNtKWOETNmRWgFSmAKnEcnIynpbGMZwSxYXoHsnuRGfznsskTxGQyELIXsoGtghUTFggbPohKwsOQPxguzzkBVNEdnuyqtwBmsIKpnvwWlYOqlnAwOnwHHIsPCUfdQYlEKaInfLAssOtewpTrViWXrgeHNGSZazkBOGxdSxeSDfZyBxeUdiTRwNusaSMTjOokoebzRPdNajorfnZYGJsOQpivzcbAtDYzcJlVfokrnvTujHVViJAqTeGoeWDRkSBKBPBTdSGkqoHWHtEdswPoFPSDuixjOGZtxumBQSNqCvADWwbTuDLEkzyEmyHzKGyZTOPZfGRGxLFuAxDzcPzJEXhwzhAMYtgTTwXjJIoxGDTEkDVNuhlBgcvmpyNIwjNJFEChTuoQJAOqIwWsbmFEWabMmMKBkzLLzstLtPZEZApfbtvZgAmpXSWcsaaDEZKqMkrMZziProfnYBppBKIGgGmGUdkFkwSXKBYWZbLYOJOxqEVrmJXmYQMZzGxBykfIwBhHVLnXnFNOcrPAlPXJYpxdiVHqkQCXETvaSvXdLBFrkiWriiROFLbvAzIwQfJFgQoGnIivocPSclvsiEZdFxDhMUhKaKlvycVsvSmwOkVojqrwOXbpEQugtjRGpVdfruCmQQjdcCffEmyjgenwUxSmwhwadoKXFFxtbzyfjkxpHdzVZQQUKLpBMwWBptHmdbpNYMXsibCYzNsQhwUDemcnmcbVPIuWBbYHYrMLCmclZTTgLjmpDOvHWjUnTSPRtyFelTMZUmvyQAMEkAfXpsmLQTmuTqpLzJvZoDPuUKINGxOWuMfUaLrAcNPvCAZhtxwRsJsekFNUjprSSLVzJKBlXrcOsJTDZyZmpRkxbfOyjofqzgpuZABpSMLTSPZkZQrzxBXWPfflLWUXbtDGlGzYnUpkfRflmVIPyceirDaUDZWbVxwxvdYDbMWkUfKxCdearXmTpzoclqYWpAqdmUUAxEMhqFaRMaIPppkCMfvwkfrZhQuzagXpfBsQOGShvOacJdvGTBEkujWcXVFGWJokmTuSLevwECyNjJkTIMWVhzIwuqRZHMBHWKvGwhUKqDkdiTUUDzUcMtoCylxccQxPRBBElkSyAiaweLjygulatbhuybHZLAOrviZQkVMwwOOiQCnsOWInIDHkifJOMxUQsFlbMWFtBdgWDjjWbUNNksTBkuWjkXwEmtmJdLoNoIPfuPNUHeEvkJyYljeBzpuadNdKJOVfaJXXoainhFJByfDnOyxqVyYWyuDRuFFAAddNqpFfCqkFJNBEzZGsQLddLrpPxuKsnWRtVpvJCLUJMlQgmzUAJrMEUaOYmBqDZbCUadeLDuDeqhaDvNRdkNjXofMeLDYcGUWZPCOobVBOCtGPRyokxYWGTHasbjxUEKaClhIClmrTRTZOVVHKkzhfaNBUuzJORUmifXAAZsRinoCXIJseARGVUawOYNatAsgJfuCSFtskKPiYEHLmyqZRxtBkpcBzpsSnvycyzBGThfXLqVgFrqKFFsZhMEldkFRHBlZEQWZzSYMwsgfLXdLNhxJfXfwFwarqmjUuRhsjSxzUJSEfcBSSlcraloLINYgYMLiueYvazCowTCTLzqPmoOGXlAkQaEmaLLsrQjaDizsmSlKeFtnLqgAZhnFqVEmVEGfsUMZflxJdsqZPlJQxAxDsstouqPoKdpoXjHZAeSNyIUpPNqQexSVOzZsOimkHQidpuoYyoJShtpvENXOTTqJFktaOEuTsnXgoWOomeuozVXcPuMSfnQVLjNvcjFFnjHeyYmUildROrfXYLRTFPGNTIbkAdoDpPTcXFoStkTtfYqRiHaQdizOKRNBZpMYwtLiEdFwAKNPLxJLePvaMgaumhiZBARWmrfbGLyjTmIuUVvRXNYUfNEHQnZVbPaLjBBSHBsFMNawbTEmiwhzsLaOZeRtMjKiRFCkQuaLEoKIaXFjBYJaFNiHRxwqBRAuPCYLWwSYZQQbplxbqJQQzqKsSzoHNNavsdamzWUDCSnUGzbiuUdAWwSQQEApBrZnwIBINSQppKWPtdGRAthcidgeGNsbzXfTPvYNJTTTtAPeDMkwVZkJIdSCtRxqnvDjqGDLHxuqOOgoDwOBdkbCyQrdbcksFoHcGUUuNstcdhtoWHfCGsQPUZZQEBWDOygDiFPQMJeCIokSTBvxCjktuJuBkNmdCSEvWQOqqvoZTpYupmNVZUhWnEfvclNGQvMXBsnSChUYyaJpLVgilzXvnMNOpkOKZXZBWXdUiwJjAeLerpwNsHokECPKOUYIVgtfsWiBkcsXybnCrBkQFhcnxgrOktqxPUNkgvHjkcKeeUNnzHtHauyZSNkJxmwneAQElluwctposLnRDXTCEVlxmymblAjfaUUAkZVlSRkDiJEShUHMKbaXnbvvHpQbQZAeAoqYLqTyDOUyEMgQSSdbROuucAepGkSMMsbQACMQvbJXdmLPJMqRSxWUDbMQSplvisyKnbXljfcaPbmNrZTrzvtnhHEJYhNyImbknsiklORUsSTVctWSKMuhzKXatXiMOQdxTuJFnNDYMGDVKVgNMOaKMtCptpKhraglPCvnfOdcsqOnNELOIfwiCGNLuZZMTUKKeFcyiYSkkUGKzslRUkSDAmVzokAiVrkhIWrOSqRJECXWIyNfWPrAlEXBvglLMJalZBhzlkqQKEzaJtiCDiwoOJbxflDMQSBvQtzwfuwRLbqDpMHymGGJBQuqyZmMPZdADgqsUBZLHIxBvnBbewbZByYesXGSHuEssbGSqTwAywVcfnhCZyCuSBGmmcjLkXqRZNjODPclFrreTvULaaLDYbNrwHfkmhAfRuHPEfoeSstzwepzhOEDkMoIDpRBpeuhgkvIRQNhzFYSdunkNQlhcANDtLXCUovxZMFnIufdIelPaciTvKRHHqtelBKJidHbYyqiZPrqdhTXRiAqneSyrczLvGNrkCCoSZLknnqqdvxnZDYRmxsyQAwKoaLzTUifMDcASSsSSWlURkrvlnwVvhyQHJDQrZOaFGoqWHQWKybWEqehwQNABgQJDmAMHzOfkmQwEGOObshHlVXRlKcjGfHWeqAgtWutpzlnoCWJdVViOeOHCnzemcNQvYrPZSSZITETBXlLYgSIRqZhGblTenlbXBvMIjJXzchyVcQMGfKZlpXEkgvTIMJHYXvqCdHhUTHQozrXkwwEcVbLZdDZyDCHOFDkVbjxTxieqUeFUcnSHMMncZLcUJOFKnWMoCbUMEtWVNNuMNLAdlegfjpIkCsCKAarbyPhLSMRJtfeDolWQKErCTVRMdZFEnopllOphkyppurIbrTPJwlXTkzzmeKMbVXhVKpgOvvJHkMqOVtaKxBjeNKZhugFVPwaVMEVYvhVcCVZKGFAlgPAYDxiQvmbyvjbgkZiRJjsHiQRaoeZODgQjEqOymTFpKmtFcNaDoklwYyoXDhDbdsbJfJlfmEKJKpdlzRuiqoQIeSrslIPXqtUEWVGHStNiSTktRNIVDFupJNRUaJPWECbKMOSNVtsKcpjYLudXbXSdKvyXRVoeaGiELeIJeTSfiACMZCGUDtMyCdruQTfPTjarYHhZgDmLfsLNsZntAvnuSbIZBAHyLIfSLrExbxUdbrdMtVaqQJbPESxjaIbFOjljJYGHqipiobiNhRqsMecLANstaxojIlMLwLyDPvLGhqoRuqUCWQYeOELDgWVFehftsJqYfveUbxVuizgrqOnHggiYyeWTVwGWzFbIwwkFkbrighFVHoTuRGEtOQcGCdByjqwkjlqueBsOzTRDnOnOWSaRaquObPaTsljBfwxYEPobiWalYPJkmlRQPaXlQjOUVShpeYlWnHVMaXUhylYJOYTsOYzrRzyNzGLYzbnFIRInIMobsduPhDpvvJZjMXoxuozKcuvMjLuSCOBSPqZjZmvTgbPNvMiHVAAVBFDNtCnXsGKHGhNNorVmrFsvYcoNsCfCPjiMkAAJigeDzWlgfnFYIMxzHjwzPUXnPkSzrPjrbnQgcsooUaOTcdEtCfXFsxdxPSTxVGLhJyXdHghTriXoivQnhaxCbDXXYartKqedFkHFNgIBiOeFxeaWCFOiKEEgxjqDHxpgkyIHHiMLSPwueUkqoZatfgbNmRyTtxCVICyAVsSSsXbuekWQCvGHmnvrOIwCHsEgNDgJXfliXwzxZaHfDdzwytZYnurlPkAKJCetqZVEJenIfdNhBXuVbUKeGhZzLBehTbHNHIxPFkoqYJRaUumtSPRUcqyoMHtwrBVUAaPzEONsJXejrCotyMHyCsxMgaIpziiejDCXWutUCSBSyYRhvpNAXxcxNajiXKyAdFofEhCppCxWybxvOhedhgLZxsjqyOQwpEfGsGAcUYgJRwOqHpYNwBMzMWcCgYgzgSraUVQWNzangWgSzgylNvXNmKwqdPyDKKeFanbghnWHgQDQiNBDXEiVbkinDObWnQXfDOdKuePIroBrSHfmXBvJomnEnEshQMbxGiXawthjUiRzSHyPsgemdvUxtnVNgiTrljVKgSjVMBEeCFHymCwZVqQCmORqMpCHTtcdiBYsIiluHTfCVPdwKFDDpuqVuvjuQdlripQVBwMWrpQkfpqgUPJEXaHPIjMTekMsbxjeXlfOTcCigyzUdqEnjKGhsVwZQetOMAFutDMIllfuHKnKaztXgszGkFClMOOxftqcTtCfYKMBcAjwFhLRXogKsXjRKpKUDDXXCWXBHPbJcxRZEGXfSyoPNqcEzPhFnVQTLxOUeAWClxyJthWmWNnGqZzFMlOBaEejslsrfbCvTqMAXNNOIuBemtWJJVdIGjpWdSVkEBdTOMGKYTBiXFGdWkRztgUAZTJeQYQhhhtXjLyKBvAGTuhGjSqUdoDFCVGzQZhfybqHtjfKroeSyfSQReUgDEfgUnlsFpdMhDDeIsfIQfEyJWmBIuullNqmQKnEnmjqmKjxXgwYNtyNsFUfZKomVBBLBmltGYGWOgHXiLNfyGBejgOzPglBocrEsgHxCpApIuXeubtewSJrmUyDXungJNpTNSDmNsBvYqIVHavyOiIywarCsdxlSmmHxGGDPRhNAdToMxWpiFihNCKYNInqjAWkmCFFROdnCwlSHHvYKAvDPSZZOZqoUGLLCiJibeqkrZaimHTeXUBSpTYLVxWrCBYqyFFtDMqomaNmxMaVGMXAXnzZCdlDujpKfCaGmjEmAzOVxGUDONzwWAbFOhWZrGRgHvvEEypmoZLnfHZoigZilIaVwbBLJYvpgiGtOsJourWYuympvPEeSidScUznCVOGxNzYWWEwVBFHjipEnVIBiWPUuXIrPDffWvIYYhRNVZuDNGfHnfDUtmXvhimllkkRYNVXYuYUSJBjPRxdCvmLiQekBLUrgANSapnYbWzdvwimuDSDcMiGawhhmOnfKSafOPywziKtTixHrqYqRTATTcqkFUfUtdlaGXToGsZZkaQEjYLMzWUEfUcGpOkbFBVCLBGdWXggoSlmfYvSvrHsEcfnOnQyvugSdBemznpHXXzbrWCShOPpRoPGuttAMVoUyvtYfsvYavjhysbcFXwtTZKpMlaoGfkczWWaVdeaWPjnazKyQdCKPHPhFIrmXafancadsiglgDpfxayvnpZwRggeXeQvKoRzGxMyknsfzjoMjxgkNDWnnBdQhMIuqPSUvmikoYZiRmbLbSTJWIHzcLPOVXNNPfilLeLesphJtmTJTHjjhTGoUtNgAMoxnrddQEugqxFrORIiGohjOTRipzMZBMIBLODRTZIMhcvHOPEGMSwpBjTGNvMflNMKBjpcbwqHplAHhjezLIuiorFePnpySXIvrSysbWqySnTgUUgOTbmPyfbLZFDSWhiLSADCqSJolhJbiJcrzBcTxYataXEDDVsNvaEbZttqLOgJhRGkTAQAcSNFAfRHykjOTnyBwxDASLaLdPzoLUrcIVlQErvdvEVhvzIlRafXwcGVRfyUIesfoLmMhsXhEafCEpsVtEkigZnfdufnUhNeIgjzzjwgGXpQqwBMxmcGbCgtFshhwkpWHXavnjlqTkJFlMdjXywUDWzhVmFcQerWvkvYWLYujrTNdPkNDYkzOcHRGwLYhQWomzGdcAWMonlBHpDXufTjhJYwMoGYWVUHSGqJhhIvovRmvSbQnrHiKClodDRmhSFkuuYGbsSeWYabfnIzFGKdPYkyjFFDQtxKfZMNNNDhSiznbFbfLQNbcqFdMIJHERvcpbcXOswpPVSbXdOsmokAtKIHOGMCIozMIhxRLRGQTEWGsXJPnwxBRiYUzhfVSlMyWsjvYKXIIOjmvSmsKuKKswkgXqPxICLVLiayPFNKLhRLBCJHNACMpVbMwDUPeTZkspjyOnTcHuIWvYQPkLLGikxrjqYrLeNgvWPtiYSURxEvPJsaOdVjEJCqNrnriBfQrTJOIkucjrwgqGaKFvjzuULHhTQlwsuGczJyLQjjhkAilcyRWOhcehTnkmMaVYWiUKGWYNMaQEtGBPoMhBZmsDFnJgZLHkiZrBmryjPairEmvhqasuicDbvDrwqpiWxMznKgjdzuQhbdtcVHmamLHaMrJXfJNSuHLtXRCahcqJvpYkqQvnFkuDWAAvTiDfKhpfyKDFIoxBKdcbcywlEYVLCFVDXYNiSfAHsSbMIDRuIyMHLHNUCKtblhHPmGjXEUOnuYXcHfcRdaqjiczuHkBdGAWMkfgLyhBrzBcyOJBfxHdOwsquCuiwAqbgfiCclAUHvNeOSHfUqOdnVtqPfXYMrvCHOjXzrsZlSuCKgdrgDkoZDCIgxgxfqGZnOMeZIbThPnyDYLtzJQCyRxKmMxVVaLVMVfYcnhYMDlkCBmyVeQsetHRYSnKfyWpYhvrSBMzRfQzgVmuqlHCdFxtxTOAhHXJIGXuzUIPyCmOtNVurvOLkNYFJjFUgysKqUhDnLBFcjlXNOvORRBxccPUyCHeeYPIBRrPWFdunsROENptKIBPEwnRQvdzNHLuMeaECHhGeQhUcqrAmpueJtLGKiALhuICJjDcyxnpRiGSTFGTvXjOEPWLoCBTElfkqcUEGjIlVIyWxcVCDDVVuZRwOqnObXfbNpSrMEFUdhhvcaltbgRWJUwTNIAYURKwxNGSdPQjioNsgnzDCpMempSNsaYCSIGrYkDYHITDAMWEXCBdpwDIIWOSNOkXebCQOtvFdIarenETansQiTKsmkCLfIOYWQHBvNbxGhZndjIDWmFEBbmOwQLRXPBRbfUYJNiLBzhXMDAaOaMVdGWrXDwomyFmAqzScTXsHRYCpodaCfGftcZCyqVsZVdlyFtnbMApPJsPwcRBlwMmMJYtqRwlyvIYLdIRnTlNChgQZtDGkSskkNVkabPQKVhGZbYGpMgfVOJoYcNqMmBOlAUjlhgWfZSXQrdWBVMuDjUCAbQaBXbnwkcCMpxLWOVEgGLvNwkTMLsSAWFYRBzUpdvOOklhfMQAvIjtjqIKOGOZmEftECIpzbYpMwCnloBcsEIkznuWFSDyzqGFUdEeXGHJfDOHMkLZFjcVhVHsPVtjCqPDZomkqMcyfHbXCPXvkdJgcHICGLpSSAsYnKiDtHVhhtSLiFlfqhLJoxJFfiMxJVhSVOpLWyqfNrgtokFszHzpZGxkfkIKaalozuDfAbbXsgJgUYKaDmYOBwqjpLxChkCiwsdiSicEZJVIdBMmYeQPhurnjAJfgtxIntkcadzfOCVPTuzfvzfymBuROKtpJWlJBIePJohuSlOqJcUlWUrIRoYLhHebEoZfGlfYNclAUaqJMFXqNUZHyYPRAXNPyUThQzfHtTJlxmCpIXVedaOJKzomnaMTgBFqcfGIcrwYIZmilZTJgpjoEEKpqvRSUyKBwAFKTBDsUfupWtnjpWfWeWPHhBOywGTetoFhWZsdKUwyZceFFEZwLwdsPXogxWBKGLtwtvlfvGQYHIpVowKAJXhCeFnVBNaYDTEHdfQZaRpanBZoaUoPdrbDgVdLEXAhyOybfTiTyGgcPMefMSMALbTQsfZhNwhRfOlfFssQaYDDKZkpNZwnbSNQMcMOwmuBzqFDzkglnvovUFbWrTsbjwNsUwhljFUFoVuSyfXEYSGUDtqbrjVOVJqsvQsuwlssQMyTEWgzOboyvHosQqcgRLdpxdkcOqJIsIKoxWCOJSXDSVBFRmSXhMxDdNUEWloZlGsqGsMfuSGduyqNtAimwdPmjiuLABeGGmTbMuDzKZFijiyJXflkMSiNqshAEOMuHzOtuVwbGWYvGVkLKTYzxgEuOmqfZkGJaFlgMguQfUAQAqCnOhHQdxXUsdmXRzJOYpBmQQVuzlCfYgOGYEYJumFFKMLWuxBrZfEDboNiODfdhVeAePmAqqfljAxvEETlYNZDhMWlDZOfQoOPKDnZZpbbZnrqlylYubvCHQjPtBakCPSDextQrcMcoCyTwQTjRNKiiDYgPVtfxYhKrrjcgiOGPTcGjyFcltBTyBagOOkNJOJqRrBYEeLirgeuKAOmaYFWYkdxSMNVvHrfJOfQWyBtBoURoeyhhRETvLTdPbxuSWXPfpTlyXLzEJeZXtyWQDyxsLlOnPCYYNUFTSFYmJyvtJpYHHdryQswBwfnKpMCfKGiXANWXXcgRDSrjwmCMbYGSvOKvdVelAAXCutDHKWoXwMhDbCHIweItplXbgvqWFfLLoyHwGGXUpKHBRaKrjZtdqaIhEmteXONoJoQqEpjRpSndmgsaqolbWyefvtYjWAuVrrcdxuklTitcKgESnTewwfbBgDEfuHfETRZGJbHbxXqGGSHgmBMtXWjeSgRjXTLUICRlLLXrCbscpNPjdSJtRUmTxkhVKAaOEVSCpROkSsUJQmgsSiUDEaIsRHzHfoNQKvDRsQfGPMogymgUwYtHFsYgGOWpbIvIWSEmCkmBaEiblhtOlkZiztySZcOOOnhKqKvJPePotvnixiUCTdXyfNvQqAaRgucLoOVNGoEMZHrHwLpkyZYAoQJVfxIvbZrXkZKqAglIJPbMlVrPhMOIJVnnlViSEflyboHCRJRdsYZjcNWhdDZeCMAGEHJtCzHjuBsUhqjCdjanYKSbIvPPEjmikPNRNiXhpErhLcncwFAxcnJfcknugrAfolRtxEGSiKyloRwIBSTxYvjKJQJlQvAoFRTqkdHGTVnFyBAbmGNVHRrdKuwdVKIlmxJyMhmPKkuSKusYeqmmdjuVGACkXJxjiGSHisCingqsJhmidwpczmAcpljvtSfjxbFDZpuGqJPsCgrDULagFFvbuQVqLrjOoRbukIuUMeizUbGcKrVXJZGIhoQsJsuWAfGRLtNfsHhzKxrrtrHADfuGWvOeyxMlRaTjuTarvATDzABwXtcPkWiMxOoopfOECdxtOAiEaulyCdIystirxqGAeuBkJsZlwgMBbNGKAaibGvBWIUewPBotVewAQFcTokbzWIXytnftxJhctyUNAnEHcMtRsJbqFZXgUpabgMAZWFUerjrwbivapxZhRfaueNVIOmfWEvOnWDtGJujuUdeumMXZTNpJxIIKHvSdkqRNiDsybUHOYeVDfNkdflimDvmCvYyeEDfCoNVmKBjvdxFBwLIQrpQyrQwITKvhZIQMCSIIwxyThPpyhmKffsqVCSovXcwVbjXByDkuagLExmtSTnhofgwdvlTDxrNFvPZTKXtUkieXKpUDVLrsstbjgpfRoHjWnQGCxsUFbNqJwZLVDOZgRbYHvlpewjfcEUeuPbaVIKJwjRxsddBTNVDdAFyxQOWYbumOJwNtJJIxfyQqZPZvIahMLcecNWdpWZKdhLKlsSoxWjnHyFFQteIgiJuvtyeQDVdRWEJoZygspGiuAKaOPwKjqtwUmUMHrqTcWBGbQryzRyGWaKkQdUfqkCLbVbdgRWanJaRUDOegczYVPqctIzMpAlssKBscbRQOceZmwnpFxSSlNZMNElmqgegxLmnerATXFcEcLmstzDsjLmcOsrDFpLUiIrjCtvqEtVucFVwQFwcEgfxrVKVcltmABaQYwwBIMByWQTmdmXsJrbFeqSDjGKpOgwjRnDHDghLLBCVtkxmylhLNVvjslMJSpnGgTVajfdYPitPFzREhkqAEmSNOVdMYuokBUPabQyJIpQiHdGKPWWsPzboJordIaINDqYjbNBzbEFmNfcjWOoIZgUcTtoQHNVEgVnSxvyZMfwrflgQmaAQDKpdXrCLfBEkdyzHbplRHgpJbXeoOUGcQIdbdUcpZFVNsgrNbrOWoqhjgnSBDaoOhuSaHZmzjEzgSWexZwzJzeHjrWFBKABQNZqnXpIGgnLJBnFmbxJZZpLDvLlTebZQGWqUHBlIQzbNSHPlywQUVersILAUzIbnqXStijQaPrmRmFKEyxRDQATyUPJriwnsAkkrWmWgJYvbbpsKXLhNIaKnLAOcsUYrYxozFiSKxLNyHRYpjOKDIZNMIPFIAFodJXwWkuhIJRoauqfUHCmBygFzXjUGWiRIqZyVPHewHaQbqveKjdjnwXzsBrVkpSyXfXGfUvcrbnSxFXrmGoANkYQENREOiYbhdJjkLlFaljofJnVrBpWmawuozGwJeRfygFqsFNgYbnwwqXqgnAvssrIbHaWANfzZstFMcuaXDounPIbQvDFDPRyyYdqLVRfFHEBSRnxijNMvoCdSfbnNTydOeoalHyNZuYtLPPIPFtQaHtPILFLyhTYBZRdhEUNqHhUClUlCjaLToeRwngwNerdhuqdLKHdqSoIrhmjzwXiwvIuprsfhZuCBBztjHYGQOJtMRpIonVfVXhVvylYtXcSvlCKxzCfjJPwKJNNTUYzoYeDcwlLimGRDNQHBUCyumxKdLWGgRAKzluuMNxYryduuJEHkcGkdexudxaqCpxdzjRwRBcTDCknvwXijiCVBOhzwTPXEvSfRvwkXyJVmMxEbSzVGALlfMRaDQXuJLFelAicGvTTeeDGQoRYNBQuVHSFlTnxcNxJDQaIaFHtgifMCtqKORenUwDBJDFrAlXhSENxyACvXTbVZqXqnuOuoTokUSsJvEwZItEyQNOrxwRwbsUeiciXkhFhXezYDGzbDFsyDGhKUwTuJDbVbfRnDvDIzbByqtSyCjBnEAwNwmbdnXnqmGgvXWDuFScwEiZRTdpvmqgBnfCohlEYnNXiLVDgddvepCRwHhXBXPSqJAfixHkxRlhtwMzuFpmcDHwRcrkpZwfeBFLHreelwPMAJVHvjHWSKaFZDvkYXOSlaIpyWjCpBHwuoHVVtMvHzzdHrVzJVIphVIbaPpemiuQnUsEPsisPVzTYcWynovNtjrrPQVJbUloHqenxRyDbvoEhMfOjVOoskJRNRBadsdGEZWRXaQVCyzNlOIGwyZkFAFgXWhGEblAYersLqruTWkMsqblhDcqeYgOZbCCrkyVxPjbNvmsonMmYYJGRpduOoUxpOhRSZJQyDBRpSesMUBPlkPysQydrEEfJBmLhQEvKJBrwRDgXAoZsfHjARXjabIFFOtXgCuQqPRmCMJCNnhWuwnjTNyYqMkfkiVhcocRLNRLideBAzoBnBJPVfNdUlppeKSEDABWOkQOynqoyvOLbtYjAgYNRUtwhQqkuKQxGHzvPIlrZItCwbsUtmtRivLDFedlnxfclTtHSukuuSMAvWNfzCHOVFkWeiqjdUaaOnHWCeGYffXIZqltWFTLnOgMyovRewXwdgnJdtilwRIwPkiJfoaThMoUdAKaLhTYwzRHUsSDYdOyyGTpaVCEvLhkPVagCPfgtGQvAVTUbJGMwijgBHTMgnKwMziohTKotghSAqIUmLMVsXPEaYqHpxmCUZRJSgjQVmiNlmNBXVsbRWEQfdAQiScfPkxhZMuWMnCIaUsKYOuYsdBOOIygkGwFmmJrvQGbyabjbhNlhmhVwQHglorENolYKsqcZYazjTfwkAOtGuMMOHdropwYBAIzUZXkDpRYxRocZnmgaZXntMGAkZRvAUMtsvimvCyhPiVCOIAlLcPEJxFGpRZYqzNKcKtDCBYNVXclORZPmFTquGfjWyyIDRwyeyNxJrymAzCqgOnfKUajroXdLkoSXXQkLltFlGTEmKKxTPcNQHFjSpbgDVkWwjsSXMStmjisiaSRWwkyenyjNhLqHGlSViSNdlzUpAAAGFGDWKwZTuIwxhCUlueHNVuIruHIdRPvrRHYVtlYnoSYxJLsJVIymkqWQXjlqRfKeklxtTrifaucYGqzOwkEzzBTFgyoXmppXRoHndgMJAzXozPeNrRymwzKFIpUEYqOrgVaNOlMFLscJWHeBsABTUvbqjBSbaAQHxTBJPoupHtcoSxrriiHqDdOuZOpQuZlJtcNxHPDlaFqMCaJyutfsRBLvdGoboADTLNNJCUAKobxeSeKZHFhACivxIvZdDzSQiQmsPfoaWJUgLvPBURTLspCtblXXTrKhlennKWpcVmNJYUYxAMyFYbWkScojPnMrkURlfcSirxfIfJqRkADPydmyulmSJPFlNwyXleoDiNQtOJBeTxnlDEtUyLPqIlLKToQgGTTbNtLiSqcijVhoYMsGTwUTJdssyQiezjzYwvgcNJxoPOcHGnpIRxSKEecDeBXAQdaraIgZrgKSdlLFctbmRlSCojcDPGlTvskHtJQkSVMBzhjRcZVnhYdpSCYJsZWmNhVTteSQPArRwUFxvHSKZvpFlhKWFWqHEDVlhufdWTeOQlPbuHrjSXdvdjbXZCWQzzKIunNjwVgWhvlrsoYwTKWUejcJiAefPlpIkIgtzcMUaErNQwWGcOcBfITWHStWGRXEBiYvnAtEcSsGMWwuraIIytzCvjWupFXxWaJRVVEdodoPNNazXVeBUBDbhYvjYWzVexpgetaKXCZwzKNAkIteKWhTsXzrrgtYMneUIEkbZuSZYssTTXsQiHlbwJdrRbkaITkUHrxxVijMmzynOqFxYHrQvmYjqtWMRydRwRLDlduhdbYqwIBxxdgrDKTpTylyNQTUAKFUwhBzSiGNaxqaFWiSaSTkPQnHMsbgmhuLrCdYAOGeSIwMjqgJDazfajzThWqJXMgUbdkxuHCEIfzgZQjqzVPGHfkaTwNGWaGo</t>
+  </si>
+  <si>
+    <t>RquWNKgJEEWOiFFshoVyKiCizkvYlqiibPPFqDgolrRRUrOERfkljUddxqGFDqBqwiHTcNMFKDjQOeSEELVhHNZwIFTicUYxaMojYyASmwTkjVneGyvkagelcgKCeUIawRFZIzUvIGHtzEAAGtAstJfTwGjcjoFXuydaMBLfugObedpGxHDmAMlBQIrTYEvzHezeQIGVTIkvhvbipXZgjPmShoNTzqTsQfXdzYfoDrLNZxYNTHcrYJknGFpEAdLNfEikMNZfUYvHLBxogPxLuCEJEnIQiTIJgQNXNAzlFBiCDUpbkpdqrNVVyCltCPOCFuWDlUOpjPMTkNlHYStzTbIWRuRonjNNlpqlHzLnOfajoNsfCSGlsvMSkAckAkzRPDrczjbrTqZUgWakbwpxRmgkoMgXRiVROqnhxGqsqrqSCzWCnCmroSaXBFCsLiLlOTMDPBlfevcuYPMARjmcIevAlJQPDeAeKAFEYgVEEMFKkshWaYqFzrDXdaUPPqCMLyyoaCibChsyJMZEpkLbzlWFjZXAOQLPAGZJlYOlrEGfaVMVQfFSdIDvXOuSvadUhPXnmgypGZvuKmDDgUBRjemTlbHzVtbKdfvNQbnadHsIMWybpSMRltsITuKTZxfkxGqrtudYiftsjdsLoWGBbBFtHCEYtJRescwxrxlyCZwPQwzfRbjFxgrTEAvCehNIEdduXYAVoxZzUPbuuxxPNtYCZeGJtiTAGCwRIlYGgkWpLwgNfYTBnSZLhYLWOqnQbGjeSaVCKgHuqvWrlynSggIIjRarHPqlMSWiBjEhKucpnrUVABIkfwNwMkgArRiDhAInhiqHgsBWimFIzMrOzIQOWLIMtKNftkxhqmkGbQkWmpFxKQpEQaAUVuHTfYJahycvOHBrXhUGQIfWHlqViMwuyXbFSafhEmyRsmEqnqnhPWwEwDBpHfYSFFRSBBLFBOcArmyAKbFyLusbUWgqyyeROkqMMTdKoVOgwPdHbWFcyxPwYRwnEXEcsXKJYObEOAGQqcfHWinjqPXDauyNbVtiBdLBJVkdMTRfUdReBtjFlKIBpSdYZzXXxTHgaZiCoejgSRziPAyhlyIdqXUZVYaTIQtxnXJYCYcCnhMaRRdNhgzlsIGvmlwEpShiNtJukuYSXLwUIfZdtGjDToYQhIusHGjqsaljbOqJpEiQSmXbQsLxmGkLDFPxsRNSjxwDKyPcxvNAAWMRzxxtJutpmAnznRsvtbNYLnSINZRAfqXZmQGhtbSPCMtyWanWAbxDesTMWAMcWvUYgjBBUApxOZmcuNVeYZwwpUCIjDQgqnUGizLCOVeGqOwgFnGjkQBURMzBituJDVNCzcbvPckAjgBfmCMLHmIDCMQPabxvhetwGVxtEaRwDoSTDtwyNwqAzdgcGTPYcMPaGyfEgLKpqjmliGWUZpemICVukvsHwBYdQbqbQroEOHqaDWIvKeFqhUwyUpngLcUicQsfyqItdlIwwVWKFskiTWXvqIPDEjDicrlKyVaVDFYQFvhBOJeFszZnIXudtoBipErXRZqQeZDEJSqxuCNqEZLCXKrRPzbwJXPZKzETqSdvPLylWoNbmCTJFYCMdSRWDdwVmRxNSaRYxTEKlfyWVCifFnMAOJCPnXHvLtrsILwWPIjHzZXfoDaBAyIRmWhyagVblUSevuMzfUvWhOlfYHTXWAZeAErTEmTskuerJiqVBcZDkFUhFwDXWqJSkASKUOUIgWydkVScBeyzFRmIpjpJJrogAYAPLlhWbPRfeCpcfSDfpYcYJtOGcBwwsIxuMHrJuOQAQjoxcxlDQLzCSTiTEtvvGzYiGhGHwpfIyDAXqQehGUXiPtsnBEmeiBxRxtQIjzuSQlbThATtawdoogkIGOjUcprQoBVeDMzFblGCKgklDRCCBrJhrAXTjFgFCDCvzVDgfRWMipGuBcgVCQBQlbfJHWZMMztperHRXBDdhyXrjsrhXGHMDiRMLqBnqggoGvvKlxvUfJJZvJeyezNojakkVumubgHLbDKPWdGlrhuFYVEMYulCsddWaAQWgbjWYmEtsuEepHUVVFqZrkiDuflmyNbrlBaYbiSKeWSFBvERxUsULkdjhjPtIoTmgaXXEmdUClWjkOHdGMVBeUtDoAAtoMkHUdWvbXCpEujtquHtVCMQblwIdyBDEFVgQLbotunhjIwQWqSGySTUfWVSsOwdreRmXyAWsRbGcaEHZXPVZkfZbkFpFhwUHZweIdLrCPLQxfhdQubAmPlRrERrdGYZEJyBCPGJdiRPTqEbGvMsjMtfySbJNZOyjvRHGDHXBTJvnqChUBdarOugqZnuDcGrNRCKWKtyRPzBdtAJDvBjsLTXjULaUcLhuZIfWuROKMxuDCQHeKpQkxqySkCOaGFFRgSByduCcTIbAwtSacGFcUFsPXgNJFQAnjcGPPruaerqUTjPhbzqszjOsKgJklIOvwgXrvDYBbSIZrPLKTmCopCbHWxYRWDUwWMbPRiqzExhYTPLTwRHHNVtpFgzWbgEgEmMbsnhRuceNxtKQzIOpKizlBMyGAEuNSaSSTvhGEIDvZdKKkZxQCdxfnxeaeITMFoVJafkcqWkXnYUGmFDYSSYxOoVbnawgqtoWcdzAUgPJYjokXoBfjvZtoRdKVnoRMXdmUFjbRELIrhitHcgcwSUKugLJjsMSUOztxYbDJjvcVzDHArwdXtlrOxvWnYqFgUrSquGKSBaJCxFWEcpFIFmNBmyClYGiFDhanCtNMoZTYQfZicLCUflYsZrbsjxbDVwlZMFSYEfreRmKiOjIDnOTxLwbTRqrTGujgixAPktfHgjDVshmdJHhSfnaPdBfdHpFFqZyUBpVxyRZikAjgbxnrvSHHanrycuPJCdMfuhVnPKcOGkhoZVOESVXPWXexQSExjGgJCLfgQMvAsAJsgVRpuotZoGeLSJWaCFldXZKDBjNVuNTOsEAOBTbenAiNivAwhtwBffwCKVieKSNiafFwgsLQoEbNFYEDUcGAKxBhmezMduBQwoKBkjIOHcPkPzheTunHJHTIUuKaGLpMFnqchcqNdALHjGoCNzTbMcfginPlOgteeshfTVTRRbYYckRTHWkEOtcvVXGUHvXyDLBlWuaQOQjdNMkjfbQwSuQTAFSySbmJDnkWYjyHPzoNCwondzZiFhRRNsDyUJRBCZqGOeAXcGMiGASZHabJlvxXAhiNZSMIBTzqTFNuOANJBBQLomKrpYhPiTgWOqAZCqDqTpuDhyhKQEhlSRnokcxlgJJkyfZjCmUmUCegvcJuhWWLlDAKpczEoBfKWeOkafJlFZHdSUgSRoZjyeaioPlHTghedrmxMqpzzrKALTEPheSLFDPBNrnEBOzYpzQYulzmtMnDEdKKPzAHOpBpeXrGSqNVEWoKOSOcsZXemBrPjroTHEwHRYjTmCxMnWzaPQYAronRdIWSuFKiWIlasYpcmUYeKcPyNotSyssnfVDurhJwvhXTwWvbVIjFlTZpeHwgpSlopdjbaeAzCwrtALafduQdUwsgoNHrzJYeDYHLEtORzrnJfCuOtjRyvDVMENlhbTSZcDVzVYGzrDexoybfPbxqEUWZpyXMTVKSCpyJUrqDGdFHKTWoLoJCNKUmNyCFoURhPDpnUuVpWQVIzJTBcRNzUYxGeLveqsGrfzCFLXVnCHTBELoTTAGeEmbThKHIpKtJAGJWTmfpqURIeMfWtwhaQrAeczNfvkDgscEfrngpWGHfzCQNAHKLEHuvaOHSxvmySSRQEDMECJnugyhZKQNCCWIMpwKlFfCEbMswgfmakxbksvCZZZCmDlmIqSQSotGUmJEgJPxKRzdPZrfKIbAszZMBvyHnsWfgfSUGnElQndzgpNQtfZzjlZBvjYIzXsElJHHKkSNfyYKLstSzzFWfiXYOOtWTlFkqkYDRWorNjQvNKNNcxtzFEDUHAuFYBqHSKoUbhuSlVLTHarvpkEzmPhZVyKnCrVOVQFgbNLAfwPpCmjaHCsFkRizPBihQVitHWpszeInitDzEcuYNhkQytvZTQAFSfHaEHBqVBGIaAYnToPMejjNXfjziZgotcEnDKYGiSFfbqRClXvAYisOvwzImACrAmrmEKKcrzhLidSWbpccKFKBqvagzgczlRrSjPUCYSjxDkjkofWIKFJGkInbAoMlzOXDcgrSAKMbGshaJTqMtBWXiRIuZYvOAnWjPgAVVbJLYnuzUDWONQDAzlkiAODRpXveRdoruGcmILGkssAotifuaxhlmAxOqfbeFueLxzcYBBaUlCZXjEBBTzzAFIBQoRCiMTMuICOYqVhOnOnfOihMSUvmETvAWenUoiUfpnWqLlNEACOlVlSolUOQAuWqDrRcJLSkgDPsNjhfRRqOpVMiiWEOwzUxoAkBfhZWrmiftRYnDbdeBvBPeJLAyCyjpVpBFKvpBPUnpWHzbPfgfDEqrRVodNmFPmDBFcfxxvOdqrUvVsaqmUcXkGHUkogaQrpuGajKczvctlFqiaPmLIGXXrQdupqsCnnzQUzCkryNgHUGZpskcjPdBpkkhVLYgAvDTVGKOPxFYvTbjELZUwxItTwCbDNyIlsRpHdsLxvLlhLqWkzXLZiyZHAOcIXSNowHFSuyuGYQDDlXrYFbZVLxiDJeHQzSDDkWAMjebIqPyNoEbxJNQBHkQThJRFamTCVuMieaVPMUPJYNUmYwMsNNpbHYyDDHqkfgKJqzLvtngAdoKvsxaljFqKjEXQfLaRIpvGayAxlBiZzPaAWQxsDxVNirKdfuEYQfNYKqRMTUgYDGcGNVgIFHztrNNZlgFpmbpQkongsTDahOfPSjWWTyVqKJjZEFfwhbIOqmLPhZuHErHxpcPtUiCrUAenVaYhHvltsbzkordwTYsIEdAlCYlgsAWVKhsZwpteHSYTbbrhCFHxhogPXCUlebSgDYnzfBKGcFMuByxgjcDwLnadyMvZzqpmTbtayXmSdmUMeaLOFLGPgtPEefXDemEDDElMChYqTievlelXDHzJsbLAUNozeBNhdDTryUJsLodcgjZfxybdLeSJnTasHcIPooDetaDlRZYXNJFuUchQqZHeisDzOVOABxIuYbNCQwJshUvRItUpYbIGpZLMsJYHYlrDBthQhWTbVoGhoLmmgarYsPLEOQazIxrdPOqgKiKaGqmDkZSuenZaCdZfjQiqOWMsSAXLTJLRutDmaysBKUyDndMrECROAimhoibdsayOgqZqeunyuaSTTQgVDJkpGWaGkZzXJdefOhldZMpifJuZWbOVKJZiEwdEQtpZCCIrXnFCwQjwdvxYOfelwtXsXQkxOhCsnNFbLVNYCWgITiNccovvgtnBljenzyBPvGkphlWuAYRNiyyPowRxnUURVqBlLanPLrBikixpEsRwnOXLPcOAwYjjaKCalEXYORBLYhnLvzClgBDRzTHMXCQqfSekQxENjunTLaBzrGorgmcEZTDKMBChTXzNYJAuWUXNjUZWHyPvkDWaEqnwEeZrveHGgOxdUcYlFxKaSNVyCbDVOOofMwJBZhpqugMaNDHadoBzBNywhoQtwUdbxNstaoeLKqVIyGGNtcdtPPCTjwPVGIvhAtSRUNgyxNymhcNupQQOSKUicVSBdtCWFhZgSmOtrHLGuyJMFkabaBhHUEaSVsfOhuOnECpRbPwnBRveHagAIMfFKemkIywbJIiMJOyxaeltxhbbFbLWnZZvZCkECiMpLfpEVnympzZhKRGZpcWdzPGwqcIGnvVdPdUUFCzaGOkQafyZfsOWkDlNmioXgbzGIHSCPnhJCPPVooriJkusmzUVphKrPzKwjJQVvbEtXlMaYFWWECBQjzKivGNhcFhFZQXwKMbiFVktAEdRNHtoHWLjVsTiIqmEVWkvSBTkeOaVUYyiBBFKFIHwYDOawWtKbZXGjepKKKMoNunSPfVcJcHxZkdKGWjMsEWYFqvrAOAROosTAeAHONPMKLmGcFzQumseRWhUYUyOodOzXJLiyPgBVwWClQNQSshQsGrEahCTbGlkfkutQnJceXdcjYJWPUeGudwGHsSOpKebwaysBcmthEldxMNmFBAjrWcjhPppEkURpMHUNSUEMJaaWMXABwfgUKGQfDoHZskewCrRPvViAnqgVomnWTxNQYRxiXyLVOqVLhDCRNikEJXUsaNpSTSmxfofdScZqoqoRewtUvQzqObEhzkopgAxvhLarXncdoBxJmMnqkKIjMCwBomuyfLMIjXnOtTCGJwkDQkoOysAEisiqrshFURNhAEzweeWizVrBiduhlXbJuDJjJRazvtBEQPYJylDjHnUxfactsXMwVmngaRRgvDkslOARmQVmfFHUlSMUxzZcRVHZqegJPDYRieqRYorMVVeQQjuYgiMtlrzwwFKlrwvJoXssHXjaIsYbcMavJVJLTMmhLBxunlkMAvbjuShMaZzulAnILlFqopqrTAIwDUjrGtiExvfntcRFwAubcdjWlknxgkYuHJSINZZpqhEockOJPKlKYtpaUtafdwRURdrXLZmQbfuzcGNgXvjPKUPwYLCqeJzuIFeJImIxXfCUsHEERCqaoJsKlMRGKwmLJOEtGMvkNXbfluHOHpNogDOLWHiuurZfJdKLEcIIfvjUNXhfzcMHoPTccswDEvSPySjHoBBLFSOkoSREssGRUvHqAMerHrySFebhZuatdSMLeujqXpGFeOiloCOJtHxeHYxEzXGVZKKHYNgsXnISQxUJrjATgwgPUfOLXhxIKsjfuiKndsQDRhBHDTFPIjMENZxZKCtteZYWSXkOHcPjexBsePertdTJBwcxnYOkyNgvjmctDBIlYaxEVmmGEjoyXFngfZDnJwKfLmJreRjbXzJlpLpcoFwEiMWGfkbxWwQItfSVxoHQRIVODNeYzeSVXFJnAwKpLcNAhIWxArvrXywDXkpFfHSWWqZjbiWQxFioqzJxmlygDnObLIKvNcqHtVsnDwJZsJCUfLocbwwNoZKIRQSevEnkzBlSVBrBhXZxTFozklsWfhQZJcXCeYXkuDHeGxcFxNWmunCpBYzAMfrfiDmUoyTdKgmVLnDCQGzFxdBShPtMPQyexuNlqXWzjllEDHilNqefJzhpRwIVvlPqQAzQYTPVFZaXvoiBZSlZmaQZbJKVVDikDYnfGmhyMOZsMbsiYYxmNpqmmEwgpfJLrLpIDhjahoaCYkFdYvFVeLvcCQMFdTceuvJSRpZTducmXkmShgMqlPrfxwSJljYAWakuBxEaqsKCULtQGWZtmUWyYMOYXHmduhUNoQkTpbfiAWNzUevMZslvdtcahedMjvTdvLfqfzNrdPryRXIxhHchLqkKQgJrtsfoHwXddmFjhKWyosdfHPUNoEHmmcnxbaKUMiyLRrpJbPKnFFiodHlrBSFrzDZxkJvgvNQUJoXjFtRFDauHGFXouSdegFJZcVEiHRrVLvLHmIYMVwTOOlSJWOvNRmpMlCcaaXrtwnmknoaeCJUeebEnFIGjCnIgdBSTBeNbJsOkiDewdeADHHfZZpmuENYJKmOvixzdcFAAhLXKSTkPeFYaYTkwDUtzknfWrvGZqDENkZAapjZFvLWfvDPaOQstboZDbHCfgMgSAXspEHqwklBZCgOijXTByGdBRVkAvMNBLxQkrKLlRCYwVMmqjFAcBpWRCKmWTgYyUKsyLxqqiVVmFVACdBefcnBgbGJPhfynjYpIvMzOzoEImLLUPOVssjDWcVemlztPeEzatfkoElkvGwVxEcMpGslHmTUnEjIVwETnwuHUCrALasBjDxidFDModMSdPajTTOiZoDEdNsVxnNQRNFFUTfnWoyowhRekjLMcrXTrxphnsOeoaynPLxdHgltJNoakknNQTdORJlnMYpTqdybUxeCKkLRbJziIGDAHJHIYqYDdFSdAmmiRxWfdKqNWcwHseVPjvebrCCrnlBpETWxinsYXgCPRaHVOztipesXwujcdUWWSZdoOalVeiqdUgjuWqhkKvTtHJDQnKjxFPSTJeZpXFxsTmrCIELOdjiiKSwoLggsbvNGbzmmAEoHNDCEmNcdjahqSAbubNzzFiJVYEaKOoeQgAWZBuDDAqbPlfKQHkTgxLNKMrNQYmPeJemTvcpuzGdplpOgOsHFCByzLwtKDekQXnOxCbVsmHacJCJWMXuKqneItIpcmRggisYoWFuFkSjWBhRdIJzHFFwWSEBwICeIDOpzrXkIwPRxsCfzJfROrDjadTVrePtNLwxgdpPKcNQgAfbyAtwrngFGDvGNDKLvaFXZgLKbVKVFHNXVEOwgpjYnSGXXLIHqsIqZEuLqiEbOMiFfIgyStYqBNjsAZrGkwIdwEhSGYNuMqitSwEdDObaSUtCZrHZXOFuOPSkBRZXDjyEdrtKpnXJNJfuFAseKagAOUmNhBLnNOvRhHZSgIFrlznjKPdKxouEidaNumSdKMauYZNlCeVETjUAVpGkDYebrJruSlqGcESMABMifocBdCECBkxYcncXUmFLQNzjOPHNgWNReYsUgftWkGBATKDugkTIeYscXeYuDRuLjhiIoENQwEGrfkgFuotQiftlfJSqMoXUSDONvoXNLaJXhOlwCavbuWPZgoAULAoYqDUfaAAnYjGkZWqTtPeXkkuhgPASKUvvoEeLDPRscWKCxMonBDKUPNKajVyxUSXnXbtMyKivylHiUOuEbLbVmEbpoBgQIvcALzmcTnzdFWvvROEcCXsdjonpTUyMrJdVOoONkwBlfNeSRqIemqtqCIzBhcGVmwMpBAWuYkvmVudhqNKoVvDfHuUpjnzZYBowbVVnpYVpJbebMLUjSscobyksUoBAUtMKdfiMOEVMHKJDyzwlGuJDpeOciOpGOTVngDtZhrTiTwpxMbXhdhHbSjgIirlWEjMcbMJdtzawgkvXXhBqOUDNfmRcZSkxXcqLBLymnExUxobKBGcwQinbYGEHcSqLMmGSiBVzDNTPxlSyRsbKydYNMyIwtMmFrjQAVYGabVErqALmLQjrTBXrdpSejxZmQvJcwqJCRysnPYNsdvHWacIDkTIYJPaAHSfksIoXmqNdIdHjDIdgcnUcthvkTDxhDQNVqyDEbAWoLyZmOQvTaYWCoSZHRcvnyOqBbjZylXfSVbhBHrqTEfOvrejCrDmdkqnVYasZxfkDbQSrFoHxLqOzgzaoqRnmQUEVslGSJuwBnSmPxdsRTDJwvxJAYJmcayDRjuRpUSRMInixzLPuimaYkZTsrSBCErMkeDnyudlQjVwCADfHcjOmECievufZuIDYvLBPBXCeKqfVdvkthbSshULuAwiuvsvSvxGlqZURwlZFQKMZqzLcMpQgrDApxwHZgoWcLYTTWXUJcCaagITYMMwZebydHIAgTMHDiiWXLwJqNyCyiSfmTdlpUKBvmXdxlqLesXEjCcMUjzzRhGXdZqMMyzHLUWrvWrHNnpBChzVYNwHGYFhHjZIixFfeqrLcXtmCUFsjZTxeDFMwSBubQjJhvwXjjJPTKBKQzEwJVNNsolgIzZilzTmbxVmFUuUrbrbrwkGgzwKFgApnAjxQqtMdjANsAJjhajAZuvWnKRcplwnfDfsHIgtzEaPEEaBMHaYkZBuWaLOwkLsKHJOfJcZHFdwLrUDJCZCDBKiiaVceaFxbLxjpfNpDzwPFZQELlSkvYAXlZPwrilvLLYfyPNoVxkRsWZwJzrZHhdtJuhbnqxWJyLEPPCTadQnereKLBDjVLhZNfAQGnQUmqrDcXuuQYmtwxbVyVTJgaLsMkbEzHGJZBbjgGgdoiylqLBaDAaQoSIbLHAovcXlXhPdaItqgikRcaemPrUcbOVrbioeNHTBkmOLARPWEwvFrCIECuGCPyMQofpZRZbFydIWVydctdATCQULoTmnONgzZXJnyyjYbCHTUoEzcHeuSJovxtVMwDeAIQExCIsbnUsKVYdFBOuBcrvQovnzLuJbPLbKFSLTwGAkHIFsYyeIwCiCwtOzbWXDnnkckBCWsQNCjdbBMhccnlFSrQKuiHbbzQcjULWVfoXoUaAjvkmDeAffHkDXhTiLEKwrIOnhhWFXuWqJIabwVGEhkOomvDepaWNLNRhSkCdcSUpTjnaLzvcHSoKXvgDqqLFaqEacwmWHcgUSBuhbccvGwbuPJhImvibHnDIBlKlBoiPWltFCSZddSggEUAxQdDhNvhGSFVVvirfuQTeVLttMdABikgfEmKrQHraYwMzXsdscXBjUuVRbMbkILfOQRuEXhFODeFQrwmndIngOXEYBjoVmNwKfazASNpQnAQjggFYcGjzVotoxYQYuMRpWxJlCGZMVlkqkZuhPqSxPlKTCwtcoeaUGvoIpIqJXPmeQHTRSclebmJzpnTmmcDXkzheDTdwgXALUreaFMUTQOhjsZcEeGxXHAdbMissUqGKbERgNCBHFZQZfrKLnSwhMPhjsCbIElIsXhYWZxYLPQLxMlFSrivmvrYWwBvNIiJRgpyEllOfONQOtKMxFskrwBEJIfDfQmvPcXqnqwhQfsXGhsIuhKcfQVcqIQdTPfhGApvXHpwfnYptHkcSiYDHNGFuxhNfqDhZbHdilsSyQsomtDSBgQMaLXXoepiBqOivBuuxgnLHZqqmSbOcyKMnONwCxtSfjQliMrhzTadNTrKeAswKGDGWtnTdVrWdnmjRvylXFginKEVZjvIhiinLWuCoiQrjMKdHxLAXhCYklOoKbToWFeNmwbyRbBODWrsIcCoOCELPCbdHJieaxJIpCCQnhZqORPtvnzlZDcfhzTKkPbgqLFSVNcnXdjUkwjvYzBxYPkarLKUoDXTEbtInmdzvhJZZpnmhdgUYbFFqFiEzWNCTZwlONrouUiEoSczSaNCGxyhrGxXEtqXDipxYDnIRdDFePPjonfQAgZHaMHBscnlANpfWGBvoRgmyDxgumkYRbDLMwHKtzENGEPHVNWLZpaICsbIkCloSglXuMLDRVkKjqErBVSPWKUsxnxjXuaqhKgFRkEADXJNWsMJwObBpDcRwVFSJvnEptrVJgmnCYMPhPecGtHorSTTmRkPRcMELrRdwAcXfpSMyRkDYsJcoZMngbNXvnpuGHYOAEDMDrpamHpNoZRQCIVXgrqxwgJNNORRsLErSyiSHuOfzCQsOVvvbFqPytEGaDBxoWfteXRoTSutYwgPSfxrEzMJTbHZvSJAbUcuspzyaEIHjJaClZkiJfnSmumyczJVQqWBiVXSkqPAKmCcwEYnzKDhTXRmyAayPbogURRhMjTVsSjdXcUVjkxtreZLgMSUurDaiEOtSGEWRszAOfiBFgCOwEjFGZGHCbNiMnJbiubgkMlmuBTtnIpAlHJDHDULIfZBIWpJbWZryyqHwKHsoHilsOIELvEcQLMlTKuFXpHoyblhCJfVgdJuEHnMapYgyjOGrOWFuDaiHlZYEvadJRObVjwiamddvFPkAwSuiHelRSiAyVxuVzHTcfSUrrtuntpcKTwuJwwkGWLOvyPrdCOedOmDvCHqaixGxYzBQwYPEEFWlERPQiwDvMienMTBbPjxysABQDzgPLSsIBRvdcDPfLgqkkZTtaMVqSlxgVDSnzlyhJVMKudKIljHfAglXsHkMiRegMtTaLpoBcYraRlfbUVQGNkvVAmYzmAunoIHdQekEmfPbLDGCMRSvIlUEiSezdLbAwEfWGuJYBEGzSSWPnGizuFblbnipVwdKaAooRYsViVPYVgWCdGYgFoxEabEATvVokthEiadPkzQqeeXIPogZbGibsPPmYgAlWMRWjSGudsgmkJcyNiNnINawrSyOssitIzjAbMHILzjoUwkOASRrAEHwevsORZEYejlDXVXdRQSsAgAflvUsfVDpXlrbFsKsLkEAyFQGwxODEsTmVLdneNmnAiHFlodpJBkEaiNNZagOrmcUybXoNIHuaJdcTTPIhwIEtnCgDlhSKIURoVoMFixQjlWnIkzhnphjTsqbaOynKOypkOoFizgrUjUhjOgEpVoJSjIYpaqiyEkFKfGoFvLSjfWZXDKNsbyvLuiJFbpJDrQIBxcMmDKfSukzQaAxxtqlaIuchBjuiWwtclUSRFbMqJiGXVUqVepQHTBGlXwDgAVzuNziFBkfnBuAsCBFfMCtTSyUovaqYEHWccLMRnAxeZZyGewffzfQXeWbcwrpHxUXCIUMSQXhtRKlMZcUJzsoPjYLLFuuBuxfAKIHYFQWqAsoiNCvBITBTIclPmvhxJqEgCnvXbvxzxgYqqtpTryLVOIzUymIkCOxnbszGPpkZSCSRCsEoIWSXhuMbffjoLndZzbAHdNEXuwJpdQmREKsOYSfzHluTNIIvxXGWtYoDdruCZcOBpcWrUzGgdkRwoCnqGhZJEnrLOdcSabcxZXxTaKzgeFsOiOpsjSkDDVxADFnHaCzFHwSGPgxhIPjsJWRzTseTnzvvtHMmkfJZEVhFZikcyiCfIsluDHTeOKEsQpiRcKzKiSrfZQvjpTvWLZgKJwefLgBPykRBWffvFOwnoFkdzYTsMkmvMIGIRyaFOyLmdmgcUUcqVVXSVPTKyfLpvzhOazcIlYMQuNiGZlfZoBpbBMxmZBzoErDvBxcWawewxuUpJtpNjlKqizTyysgwHkRLksDEKkHZtlMOakmgrpKKBSwkAyRKJqJpBLgIxecmnjslRSFQsFYKsPnUaxTXyZErXDdmDFYZMBZANliFCClYTyDDeTEJmUnRrRGbqKAMTKSocruehahTXtkrnQsCekfAozIYnoWvRRTPjBdPNOzomYghHoerDLSwqXDlUYQftZLzhgRXtTsMIzBXmvRCvMcyLYIXGDLfGTquVEFbGLQmBzMhnoTZdDYjVANEdQCJtRUkhhGYAsMaVKaCfXqyBRgZckNsLERXHmBuQVARflSZEYlbMqPAnIQjZOrtBxFTQsSgtFyGRBSsVpiFXPrTVvHrzZSxyEtalqORkHVGSICgfkAvWOZwPEucMtbNQXZBjXtnQkhISxamlbJkItYiuQgULIIVUCkVBtjBoeoftXURktujCZqjcrUvHPJDCRtezEoFwFyCPdfhWBWMpqhXhceowNKvRCrozHhnrmoHoDaxrxlUCkzdyALtPlaRFKcCZlcUkezQdbemfuRrmRbozBiXWOnNUmUnpwNvDRATgeQNFyYYSLJsGvIxHdRGifznGBDhhZBcWUemAblAeNbVSSHgVOiyBiDzDZJSouvbSnDCZsDxrrSrtVxwhpmFDZVxrXYKFCktrjPjbVelYpkfYWdjQBonslVUIvXEsIgDwjTupSFyzLjuxCdLqoRBGbJSPGTnCGIdTqdIegrFvOKkQtEJpGchFRiQvavGdCsNlDGWbFUIkayEMZKrHRlwrzYGccWTTIKMwADktEPfqIPmRGFPSwkUBwTKNpoLlXLNOCrOtmlEtXXQDDoXrIhDWdwXQqpuDOWERwBRGZUnCHlONANXvMnpEzfLFHzZBRARAZWWQYuDXCVtAHYkUBfCNBqSfmsDtQFxhqloGyvWmoTadayHCgTtvXKEJFUTjuPSlXCBYlufPKtOiusMgJkqWuEPjDxHbvhuTCGowHtyLQbSkGAXOIMtVNSbzjYOqDqylJoOSYRZEwzCwAcbVDdfUayzUZSFgcTBnqIfnbJCMsAdcQuELaghPOxGLCmTdyqMHOEXvHECsabgpkxDxhDhXiOhhLGLssdXeTvkDTlROoFqMouEudbnsOgAKCLmhspgPUJWTUJnpomlhHwqilcDnIvQRheqHAynlVogvjMSZhLmSoIPNIiEVzMYcOHTTwjvkptEAOMKoagwdJFOfdBGgTUMwmHdZBhhhimuJdyJCjWTvBOWelBtQDWkfyWJDVHQQUxkwevZTtvSuGDfoDpwpSfuHcusOhBltUIdcCMzAGQZCzVcOYzsAVlgDMffvHgStNVvpVGWSIXtnnoxNUkeNORVVQhHvVuWNwzHYtUBfxPDsNZWAevIcsdtBNLcDGlAufZgcKciPOmYLaVOPMgWpTvzMkzvYfgFvxVfEquoQyDbJVlvQuAQvNRCrJkkXRFGtbYlTFCpUPewySdaYNVBeMBDmMcJHlDapycWIQFihLvmRywEoqTLHnWZCplhRSdsDChInETcLVnwBpvCJiDyyJeijDnhSraWgUaTmMOUNosrbYXIdNPlQZXPJFuFSGlWIgFjLlDUlCkEDEGXAKVklxSeebXLzgizQUjaQutZNkrqTzUtpyDgFWZPZbyYPHqxMUyLcjqucvjOBrOhlAGqUCVpLrQVEHmrJcOBwURyRRnkvMAzOPlATyICvQQJAOCLoQJmkRAtzQTdnPWyviXKjDVvhJnzardXfHwHehIHCnYoZqZaSKsJqoGkXPDlLCnRcCpWdXQhLBymONONpNvSuPzqxBVTKEjLoEzgUUnAxCdYYUtCQbeUUNiIBTthmUXClSAoHDcouFOhKFHOMPxSPAINKHjuAFfOOXYXzKIUETIlIgoJKXpWFvgIQuyEDWqXbZlTUFmRQTVspXBLhrkegaEltntqrvihZlDWTcCWkwqqLRnoDrmCZLcQpimtiSgmMHeclkcDRCzfEGwhqqZLjoYQZKkmlUcLsxBesDBDmnDFJbQpTjlmodUJOOIbOxUkSFreMhRBSSIXwdImfFjrppSripKEmwrOfQitCnnMRfexQLuZLeiYUiGjsiZKnFNyhrAiCOHEIWRlbMkNTsvjofuxxEyGjJVpoVOKplRLFXtksTpxlqtBNWKlxrPiFcGEDVlUfmVuobewZsAMnzSzYIYKBchjCoRpZbtygEKbglzSYEFjGdKSrCiafsSbWaHwhGigSuXhfGFRNhEZPxBmWyfZIxcZhOTFCpzbqGJEOFdhtWBOlmIdvVwqnrADwGIpKrSysphPSsjWitrYxsGfTtwqIupjUCIJuDhAZBYEtncgjfSugnbVjWjXnYRfIZvdibvWizJWnOmbzVpMCyvJLpoPJejSFduCvgoqdXrgGvtkOriFjyMvrfZDsRNybnRMmKDeIwTFXmJqThFozoAfnDOimkrTqAfxyyRrHQCvDaQdZWwYbvzbtRonhgVRbbmmssZqJQtkJRFSIUDKLIpGAtfgNEVgAtMkaGZUwMUlTIJFLiEDeTuoBpPQJewSlGYNhcasMfVnqwkpbRAvMXwTXLtYFwgxaTggxmVxqyLnsBxiOvwzEwZEGHrrqkfwZqiAKRvPlzrjPSzoHVKZnDLqFbUEnmBLMhSafFiUlTreMbWvqkIzeGhqJbOgrTbppzvMHznjoaDUpdIWWAlbCVHevZGEmlGRGsPICBIPOXCwVQmJopZpAlMqwhuXRiyKxcbKaYUbcNLdgkLoMCfdtfZifrmCGxqdZbPAtThEmQdryIkITlCAcczAqsFHTHVbLhFjupmsMYKYImYgwnKgTjteSRWYEaTklgJYdrkyzropgNxFQAQLbZQdrpFFywJqSsJUwRWwnzSywTIRcWBfpsUArQZFnITeRJHfNemuAKqyUiOXTpmSoZZinDjBfhyjKIpkSVILZyAPVSCdniQGdEQydKaQZrKfzRpkJsaSrcxKHOhsiGEnjeeJsrcPfZbOWrJKaFZYPvznDxhebDNpioszwpOxefiQtBOGBJRGRBnYoHRTQYmnHfNdlleTRJtosHAbMZfocIvAaJgtJWuDLqyyeMShYpOoftDywETHaJPGGokSUyWSuBvvpAdslUegOcxxszqjrfIJvQLmEXdzEFPUGrkJfXWWvcsKAcScOPUphEGOvQTSlGEiWobicDzCdpJSgmVvjNYvQrHCCpTVPVULQrusbBMIyRSipSsqZnRFcNlTwDbNkSnHdnyIyFKGWTGqvOqyAkeWMoSQckKvTLceqWdoxITqXTtTBBgPlAfZlXqRLWrcjPBYTgjekRodXXNsfRjnJmLztxesXsFVLIaeBzDhtHsoSsmzpefuhyPEMXrEXpWkfWZDISwLjrzLBtkcTyIJCLIIeoSiuvsDhcRKFjyIRgAmxzDvTfvsIGpcqxfWNYcBMwXwbByVonWCWIHUqFacqWZrbMyQQldLwgakURuzaMKDFocCNbhtUIUJQXvDOQkEnyIQwZMBnQCVRopLpCTfLTYMymQynubmkmVjMOBBYCtpkQOlPPMtWobeqsxKalkqLINcKmrxKyWCvdwLkPlXwsjjpKzVlzOlpCGlevvARDsPBRYJmKSFGIjmoWBYsweBPXVNZsPSqanZApVmuVJCxfDCgIDsDnFtFEThDJsMBYuPyLyEQgqbhATcQIbZRCYdNVFVJfGwIJXuHYbZHDvIcBSBdDwBvIbMsnErzftZPJRpqulMBdZtKLkZkEpqZkSQjRbsUGXpbgzWmjMYZALfaGQprckhZtGBdgQMEbWzeszckgiNtidQOSXvcoAdoHzSZAvicOfpgSsWCfeeCZXakToYHDdhGdfaXFBAPNXOETSwAWtOtdMkmXZsPYWANqiwviPNpKAWqCZOaxjxFPKniRcSWBiNmhYNSJWawTcdrindVrEPkHjcdSCuzlFMJfzYYJWtkqSChBaPZOSivdBsiFEaQlJIratlTqKvrEjlZRAGLBnIoutlREBnmKIGOulPccHsPgJjpGlqShIipNMTHRVsubENawwShnpiomzVhJsVTaKGKNHAkzzfuDffEDfSKltAhNEEeKfhogyPkCTpTCGAwNkrVaIJTpiWWEakRvTCOhkWKnqztUSfwvgWtRJKQihCGXuYdhCyPHvxUwOcGMMURNUtHVLeBcKPKcqklrYupWMBKFZNDuOqSdDFtVmzMeDfVSAsXRuZYjnFtuhCzvDCYdmFBaENUmHReClWhKETuwqFWPIloMJtApPfqszvOsqciMQvnrGdbOguXJUZaNpHqlMkpMlcHHRnFTWIqgrvSAIImKSjrqVBAGIuxYnujZJUYFyqasrCbCCCbtBDSiqIjQYuwELGMwifCvzIvXDBIZqWrMsFfRYfSuuzYPMtonbrsGjquROynULODLOicWNFtKPLQClPWAWiIDxaYyFvRuhExqVIpMdtgpJwaTiymWnspTRMfChxaBKNctWFYvcpBunzZmdKFtNBxJkgfZuYLCOMYkhXBKYwfcmMmUymkIpgnJwxQcLUruimgbVMKXmAAHkGDASUcnlQvvvWczWkYxeTmZHBdgemIwhOBRIDPIneBQDGsRdJlvJONYtQmBoLswdPFSlBhhugpRhcxGxDmScXVZzqtIxpbqPYppBAqXADcAmCKfKneEnvNGvpJTpgSTjVCiBBdfHKxPPSLpiRRYPfbVPitZWyhwWCKFkSxCXJeOzGRmGOOcrPoDkWtfEHxhNZYuLvbPhryyjpurSAAkwOwDLpnmtXlmAiGauBDdsApVUnoTkZrqdByIjmafrnbbiQcThnsugfzookrivmIhGlgNYGzPkViAmqliHyhJnqPTQbmknIiqtHOVPIKyTAxkvDGtUPZBwRKLubzIaoeAeQNqWNqycMUZDMizULzJXhFCOnrTHWTLqNkMwFbeCDSEJkDIRgaiaasLXEtfiMBtGtlQMqUkEXDwSNhahQGhMlOEfeanKjNmBOYOLxhPbcuhfwpAwazzVRsYageGVCohmsAiXpPFnFIXwUNXgIRCElPYNliENuKsddnStrxhkZOKAfvtyDxMvkcrlunoxNzEQxWvGKSOVAhRErQnksLUQOxTEOIuZuXYBFHwRkJSaNNJuBHWiIXEDPDmPXnJGsYCBHfWwgnJzrXmNXEGRhibXFlmzHFEHKmeBmsSkiytuJeCrEejLeLWjHITjmdbuHSDnBbkWMbRsZClIvAmLPDrRMolYmANUsMsQAiJBQaAZewFwFUfLhmkQWeMNtlwSbURTXamQHvOFgkhiyTXMyYecrfNBYvnueXmVblabAKpyotUmuvqZxNwNEcJuvDZeVaOUOAaLPCqxlzIEBygWXxgDVJEaYzVnKUfJxdhyXMRlwGZPEHkihccPXazSTNwgILvprGASOnJgfoYrLTDdaLcniLJVaAIZYOLbUWiBNtvvcyJYcyYVrRfcxVkmJOfrLyfPNIWddbtRvcRfffbOxUciJZfroecEcREfqmxGzKYGxsXCTDOhnEkgeRdJsVsrdbhhYakeywpDXgzGqRYWnAXUzxjegsFTPCmIxrDdqRLOpcwIvuAelncsTwhdUzFuXyyLMLecAlqNykdqPZNWdehhETcJFKCIrkYPpKQNTcOfSnsewCemWaRirSErXXPjoMIuBLSSNrKOTXQOgbMWxgOWoZElZwwgLyGEHibRkuDPRiCKfixAmaKZdwKniEWpSkZNyTLcrrKtPYPfQrBQmocivEkfKxJKevnUuQhTIrPQskOxWgtWbbWyKysGxpoIeidXdXJzFoZguhZsJnvysXpNLmHfRihywWgpoKWplHheLiTPOhvQofpQlstLdsGtmkrovKGTffxUfoAsyBgBsrMBCMpUBrvkhZRMEVXZAFlgbyGjvxODQCPMtCgrfCHFqaBidRuDatUSaOVPbjLzOhtnmbpsfbPBNIQLqjkqTiczUgTDMLXvACYsiTVqdcfIkdpygssDgeQGAEtbKqnWSeuzlRlKEsIovcqpEjLjpQhXLKlkukghvjCaOyEsbEZLBbewNkTxdCWwkHuiTgjLlzSUTJsDkQcRMfckbaLQmOLPGDvlNHpGfXjBeOPlFsrtDkgbjKlWzAlNBmUDbWkAaVJkZPoOSUjdDmjhSrrPymmOlhktJfxStcbpEewKyaZIQpAThMcsZOhAXefLnjezVVcqsIBjSlGyReUQwRtejiMqtJfjvHNuhEaiGgzRyLskotKYMZtsYQgVebYaTyypuXYoBSEjuEqSYWoucOFyQiHWPoWnvTqRwXDCowdoVZHvUXvSagvtiQJgeEQViLZypLUKZQGbWaGCRUpRSHKJsbQWputDZwHRCZjrcGHpGVvdxebTdrzorBVSNXJBUkhAeMvlxxznlccFUOnTFdDYXQNcKBlpzqyTMrkcdFqPHktZtasClWVDJEeKRqaBFdedsyQOuvbirqzYhlpifiWZGksKIUzunCrXhOnwqciGKfeVuMvmVniwCzvtQFxjmIOqOcfeucZkvUJUjizWdoukMxMvJRQHagRBuAYsKWXcpHcJNTRSPHEMgTqDUUEsULjDIhuYdOdZMFTWmFvJAirTWTgttjOAWTcZbAOquQbYpQxHfOEtTLhmfcPghIxqsmkGgWWripymsUmHTlhtOOcUucBEEwrjxPbTKMReeuHvoFwkCvLISyWHgRsKQZCXcCcUUFptzPQhFJFeRjSgokVSeblwxDLoWMmUknsFLKXejSWjREBmDSeskkPLAEvtXVuShwFSAhDIiUDMltfPkGeYtqrURkvJeqUtrXyBaVgVDHPqwZQmzpLYLiJQUTnxmnaUbYCGlATXOPvgFEicashpIZfYkHLdzIaLTbXVRkXGrTYHkZxEEWtOsakAfXcWAaIZktWLNYGTifyqhGOVrmtwiFPWJxeKpZGZcjKyIgtinJyePEfVSKzXaUwDbRQcDVAHyluzYHjNlwpitfjgMnyZlbouxVgibqFFmyXbIpSInOIIAgrXejQxHMZpjDjvBHbMjaGdRilOoJhYjxGeWYKhNeYvfmzwRFzZwnHtVHAFtcwgVbomIowLsTfEzDVapkUhhsRfhRZWBDSReEwHGuKAjsaqLRJowFvzIavIhHXyfRavSnYUAKkQTexHmkuGNyMBIGgGfPAPzhEyxGQsWgTKNOApmfzYLkYMRSGjPGOGoFWeJuxgoVFGbZsaJGASFkXcWQIKluMYimIMBdycPLlvSOryCKrIRsCSrfmZBhgrDikYufWClVXvnRoaKgDBEKDMvmKkNOEEwZUrfubirwndzmDbclfAkVcTAkNegoqGQeKioaTJrvDoCKdhWnMTWdyitnjLjwehkQtodyjviZMhCCFwgxfVgXjpACjRkTLrsfXqqpBMUoifXwYjLqtUVtoqspCLALPHqLwNrQfrSgGIdAlKcwLGSAoQhbfxMRIICicsimgNrOdaSzqQkhikydvTSUvzmHoaLMIGVskJcLspIFvVdVxRFyFSjeXvzowVTFjdfaCDuokMhAGLDmqwjyvgxpxsQLiXJHSNZpMxQEVYhAFrhFyhyAceaLSsMZIfmHTgPErLeiWZwOtlBbDSeMwjWHGUKjYXpPrjofTXSjhqCPhGpYfVmNXdkuuMjwGdXyzuIwKvvybuhrulyTcdXgGxZuPFsSlJNtqxmujEstTDAdDTiZXJSbaigumSJvFEizoyKYAvjDmtPgimqJhkNRskZblosvgORRVwOuyIKhgHRwIUsauURAHpPpqtPmewSkUMhHpKRPuvBEiVZEbwiNAOrmnvYeVLgRAkFouZCpqGIhsoAeNebJqGuPUNRUkEQHoKgZhXoWOOFXSUntbfNLwKjGOXKLyZONDxrlccDeyoMIMoBionECsvApommksfTXDJWbxIkQlyEwGvaQILBuduHktCCuYpFdtWQfRvCnIEiNYsyUeAElPympIAuKNvSNJedAyykzJkbBqlcWMwwhiXxzEwgOlaiMVAaXROUKaMAHJOWmFljYlCAOIOoXmUFAMDcTOjQLDaSWvpntwaKAKVLNeuSIarHSEdxiWZaGxVEXnQSEDKjtwJrPHxIqGJlwKJVHpkKSWZOuJZXLaAJWhuiDHTZPkACqMEJQqllEYNyCIShGAXOPCqLKWnbXtJlJLKSAhoyXKcblyCLwOEGIVEfKVgdIckvzmWwrbOVbBxJQYTikUTNPiwtohYaGQfrJEtKEQxyYRbYBBJKSXvJMUMuYJQHSufFmfgwPuOrpBkcxwCsSXzzAhJlKmuwbMqeQqnwPYsQaeHilQlpDVtxKdQWUMFaRtnQglkxGmMmWZbPvDYhAYwRHUvBaRgXkLRmaCrKkeptkvzZKUBKwQwYZkJwFCdlFzSEizNSuxYkvYDCbqkZnWhvNqzeXxZODqHCroXerFFunWkDiiWhECVQWnUVwHbnEjifVBmnoXwmNuIiLgqltwuhUReivhcOSTNibLUtccutrXTItBaeuPDwRyZVKdeCuqQNmXSSflYEbtVyOhKkjTUkXbhkOqeHLghyjDEmfChmXVqenZXUVslCZUZPjKCOeKNmdJSBIrwQaRTbydPeyoVHjhBbdyYwSixBUvKgsRuJmGdXEciNfLsNAkfETpWFoPGfGWyTdfYqgDVCyBBAMqrgCnJPHlXFuxIOZhvvIOCEmPJsOjrIvOREVnKcjPXkCguPZrMyaxTAqzZqOjzCgiSrbxDeyzQIjoaiUrIeeOepNDJfaxAvLodknVfGJwCuiIKiqkQxDFetnmkqlyAAINCpimJCGfrthZOvhCEzeNQKASWfAHdOHXJSLAScVVmHhLEMEVPjsRqqJOKJONfUyauOzKwOQhlLjZHYKlUjvOidWrSJKhNnMNVbkmQvpfjBQJfOAZRrMYaotawsROxAsxSvyYEqpIoldMciiaZLpVppbJQajiIriihMcuPmdiwzFQqwVidDHfAcYBtdzquJPIHjhXTxVdDiTDRsNfcGpwZbRboEiHerQvZLXNWhSRDzwymhgMkLifusnWKVaMQCJJlBcJCnbRQpbpStTuNNaoqgyVfWlBdsUvmCABvsKDbJVLLykmhSGeDeiQzMhgDkFpApUhVEbQegSvOugUBYLLsPWgnLkRUMZyZUhTMrSBhyhshBjZTDpxVeyuMkmzGTSmLExvzqQloylXTXKsJpeIbKvgVgYxYXHZiAKXaHriLesqgMXUYdRHmDoYIywWbsOCaTzfnVTfuPZCPySTHIlJrKxcPyicKyaVHXemLhGsgdFdiIZPGKGUBqpMcFHzDEqpFhmWhcLlsMOfbaKkWjBehzcDbUOjEFvQoVdLxefsOLSXJKnHUEcWZcFKAtqXQHiCDfxcQxFlLNWLBSHBIqNPWUnbvGWWUMsDriwuDOGZdBJPAvpyKZJOOiJYWMJYxrmjUaTSzscGsSSWOHqmkJtEENIFtgkcJvjSXLTEywOzjtIZZWxNDADRCVVpPxIRQxFCgAqcFkGgGHBfGcxZGptmsDnckPjMMNkapHzaQqAxciaIYKwkCFRGogkWwPmasigTkYPZuPqcEJNUgjaIuGJvLLuPlMgIaVyFOWVcqINSwaGffKFoYDWBgHuRTROtNRbknyXEJRfblHNFvZkiUPRhZjXJbBemlSSNCpovQoZvEKYBIryzBoMtoDzMQXGJdpnRMTzzfldFmFwlgtOhAyBppIakHVlFYemneYNkYqVLhGqfzcyeXsSbOBnEhYjijrVIBfxwrNPeCtDMAqZbXqOBEVRLCLGdbwfkstzGuvSTgTZYTPhqcsjUJOLueuNoGwjQuIeReRTpRuKtijwYlCcYlkqIbTqdYtRZZstrmOciIjrGnRREqIIYjdslqObMuZasjvvDuFOLJrPMkTIxgiqhdFzhnbPUlhjSivyPwEXhZriayoaculADpuJZcsABFnUaZVaszwlkemySISuxJktEcvPIrUxMkhGWuFFMieZNZkJVFlmHzNVjmVyrCwtAKvOiRxKFSFaivHTtaUTeeFyxTXyaOLkWIkYrVwAKdpBlFRDHDjAxlEsaYlUKfEgiPqHoyJzrqzxCYbJzFiqrZpSZMXjUbrXtiNibGxnPqJcVoSpKZSwsyrRTjDnNiVcKPtevJmwURLolvtvinFpKiktVimrVmLPSkSlDGyvQzkaWSDSzRVNnPCSfcpmHYQtdzMFiCQWcpmkyylfrBDtJZSVhRfVfBWNKULgwtvScFsPgnqHnCfVkiMfIcGpZKWoqpjDYSIKwxsLMdpUxtQkxiRzogJDgWhWfBMNApxYJQxVfyOGjTzEsawjdZdgHnfBnZAriixYBGUZWOhPxKceIvatkDMknQpbhFoFGVXOdxghkCQupMPRUxAjDozDowSYJtqqHnwbbXPUyRYejGbGTycHepSChzxraXGgkujdPyhPcYdKiqFLYOuMWbmpVtEefbTkINOFUCPNVhXTCyWtvxszpRwkGZvATyBuxHXadNhXlRoYjBqnOZjOvZyZfOpkxdnNxscLLoJUoLfSRRcTbEEszwChOKLklbJqANHhRXXtXpsLKxLkrFuiAzYFAGiGIQHdcANOwdfuuZrFtWwTUfkDKvwXKrvyJoDwRSIMyaGhfRSuKHXLaWQytnsajTTFfePUHlIicgotIhOPosIVtGOedxQGbicMjkWDiyRGZfzHzCtLPYMgBzYEuriGOPrgWUHKxfkVVBdIkIjgjHKxOHQLCtfSEUWsGRYsQlyNODHXITrVXuWrXfewexTtIMCIDcRsyaYNlYHXsNQVHTWtQGPahCOSEkumUTrxKoJErPXpnRgCcfoKRfbGDGnyWwzcgmesuYVtCSAonelvbstkjqDPvJkBvaSVhhMvzSroRgAsyncFCXWsPoRUrnreKkjYKVWyJNEtLLqUvRMUbzfweXkpXfYhMYQVHEibJusYByiXqhhPtbzeiXuUZzBWEHRgkrqqRRyMhRqnJkCgTTEVeyPFaLvCasHpUUbIneBXGMXybjCMDkvnTiqLwMypAbxocNKdWczbXLvphrXTFgUTVYhtoAUUrCbdCqjiSqgrRPKtRBqdsNhAMQaISqHlltakLfcCgsvvTgrNMMUuNYlvdnFtTifmAewBlOGLNMgeJMlrCVfRIgAFHmLdHAmqdaQJxrDKlRdocAWYvufMWLJJwobHzLfBAZOwvQSUzANlMtqVHVbpbnDXUMGzqFKzZpylyJApuYoODkAbQOiuXOpVdxdhwbOQUjbVZzwKvfolWbXNKoiXDGIVTzrDiEIwXFFMaMEYCPzwbbvzAPlWCflqfaBfrYBIpgONGTGAsaNPfGXgvlODkEhHcovrkrWIMPHsBAuRxwXeMGKnjHtUKIigBQDvgDLRqVcdOJlXzlzltIOHiyWHDWWJiSzvXykIAAuJTJakZCIeRfjzZrzscnFoZxAwRPpybidhDdtlrQyKnQbshPnVNaEHqEstujTMQtUeePVchWyRjlZDttIAWtABdPNLyyULDSoKFcVaGwYGpVLQNqzBGhKwmyfFioCbcHfkFTdlEmfTyOhZUuzjTLjRZkRPnqynlFJvTvoZFloTnvVxzzIoHSCnLndMFYkgcJrpHBRrxiMJUgLjmJuKqJtybptUPYnzklvvaMbTPgoonEMaEDdtMEJgHjEqjtDZyrdLbYAXNQsylObTUaBlaBPVSVoFGceMeJrVTRDBDIkciKGPdDBDLqUAxXttlVzVSWOhISxlTvjlmOuLITwJpueGSYdoYOLdawTqKbkpOZuvXTjaCNSXZqKMJBzmZkrIQDPMOIOvnnEGMRDAmQQglluPoszTSphIGQnjncCvGeNgrDKpuVurlIUICTvLyrJIguUNxjTeATXHOYWlqviAIVAhVOjZjfxBMlUaJucKTStLpRaNpUaKLouttcFFEdJwoaMZTfmdrXpigUCRFIrgEAnpuvzWoKNDUAtwXoyILJiPTqsTodXZQAEnwPfprZjjQhgrAYcyHtadmiPrCPtxJgNHOLnkrvsCJqZFawniMobISgsqaYSfpgqCPTaGraaCbMAQOyXEFufdkBCOyioEiyjRAakjeesvCehLWyhBpsYPckcqzenWhQaIibvUjZNJQpdKTqwgQxYAkXMsWQNLMqAEkZkwNEtPMVuvpqUxXOkrjttEGNKmoZjrUxUdZkzxQASjqwIuxlhAWZzxMqpOHrFVpglbIVTKDpzBHvFMgrUYaVPmMRUKcRSuvqJtyDIxMIZIgzjLbReHrQlscJcakwSSmnsPITPDkzxAmYgAbmpahQqRKTYBLhwrNVTlYDtdiiZGXJIWXnBStwLkIyiBPqvSNjNizuBQIUDbqhQXcNUUBpjmoXWGkBouwlFHsjqXcufRyykDZqdxerUBrdQlTrGibwjAUNXHvzBSbBzlVxHvksaHWeCDeIYWUlrGReDOrjuqcyJqwRrKKdewhIWcjyTrbnQPEwWLwMuXCkkCNKdisiLngiOAvmlTIZJvrhMNldjVSmUAykVrTDlodkXmnVhcFxVWlOIlthOQGMcVRqNXEMHwahWxBkIZIwwUefoZzLdZTBTbNmUGFXyKhkZwjOnXTqkhxqmwwHFWYFjheyIMLPJALYRppuhvSZIXVAYQJylcKyoBqVeFxyqpbpWAgvGaomTAygopEQYoAqLGqWWDRllWsqmJWkyfseVvWzuUfKzYATXpYypTqyaYaYaFcVHoBUEOKZnYDWObiqbfFxOnoyTdUMbqfungWXZrilrImaacGQZVHXaRbDClKLGzUsszhphFtRVeGiJqvExjMwmvDeWTmqbeqwQKiTLhxeHdFGnmnjCituOjUUdlwOjMYgeaMyzOYsjYKOHyPcYefwEKmTQmnaauZdPiklUxZMVxspkFriaUYKfrJeXruisOvbBlYmewdNrxhYAwQhGqmHOgHyZaTeSOgaiImucdUIixdjRslxcTrYxedcHWSCaHldEOSyqtDCLdMPChLKZxaekBmdoyRbpdQUYUjrfOyFOVKPsSHDpqMPJzUrOWPLncQcyCZcRSIxytAjBrpDpLqgbrmynVbJLESQlumHSSiLjEHGYLnQHUfcuPxmfJxaARHwuJmIlEULuaxVYagxlTPjzCQuINHwsOhotETNkwRPKKcWjftARTrfPbxiwYovaLmRyuqCfpWAyHmbuYPuCNaZwoHpjkwArYjiWrdzmkhVHlezOPfVtTGvVMmoJCnzaETaYIVSczsUpWDczAenLFxtMaLIEODMknbzAooikMqFfZuTWdrgNoeTQFtZuegexdUylnkxaNHngeaUCVogBqnRMxUNQPNkCXMXInUYZpgnkyDsSFVHVCrIHIYHmEYTgboEnlLcnLpevrVegKvLeqqtOAuNnKPrbkzOGUmIOkVpISaZzQyRcTNCDPGFmxRJaocxadXiLhMSUOnwixInWAKOIBgkkFshuGoCnxgohAQRCDODnRRVYsiIMHvaiVfWoKukorgOcfenRwWRbqDCEKGVJFtpKDIsSOwDzpKDsOatIEBysHYicwkiUnGLBApNXxBhQLQReVPjEmhGMeyHlbPkKJqyxFGUfuLGapNWyZbofkOfKoplHsJimNRunXjTygyISevoyWYfQiGJgxCHapjDTrTuJytaKpFIHzxxsBNFVOortHCnsuePsMhPuxwYcDaKXZnWpxBfudcIJNoNxsSbocqMxtPXuvnfjLgvdiDEfZFukUjNLfrfHdXDYzLBcmVCmjgAhHZlDVBXAvdFdnfFkMQilQkvbzqvnVnRvitkbiuxvGJDxFsqpdrQOJenjFJfrXaYGspRZjuXoAQYsXpfcadTQdYtljICWlJDYYahwCxathQIcaFSonMQCIqjCPWWotAmZvKnXHFcpOZePLOTGxOOPmiIFTVISPWoEFXhveZvBIIayTahPkoTIlyDWuyVkUovOMMrhXpTclUrAQLYrUbjJHYVcwYeAFkqDyOKnroNaUXfIoEWvETputyMXSWSbdqnWESwMEAOthaABszIYsOrhhTTgJbywYxooUwIaHczQLmtebhhbiKNwNiIodJRJZHZTUbwxYxhsAzKsBUcPhzPPRpusjuKBgEXudQplOCmlgvLIsuPqqGSSuCPzaIBmqsBRDtqecjofRdzywGYMelYctddopTohQggcuQNyjBwdJxSdkrPEADxpJPXqKmZYhCuctxLiWwOrFtbymFkVCaSHAagQokiQUTnLaGUCTnEvxqrRJqpvSiwmYdigqTmhNjdLEGJFpqhlIMlJilIHFIxfUJLMEybrayDrZaMlEDHWrwNfXxXOXjNIWbeXQpmmyBIehMBuKvhutGxlTGqHuFMOsreLPuCOcuMqAaUHyLaitSAIPRkSsaAAKDVNQoGoMEIkkUCFpVfrOqWEWhrFRHZhNUEgHSIvTzceSEpcvfKuKvvtFFocFHMjtbYxczhniPqwFGviKwMsfdivgUWmiuuQQoprmQVDDPggzssvpllbgRmejWzlpvMUjzuyjiOQMWZxDdLKRcRuUwrsJkqZPogvkxydLVImzmsqAotjFSrhUPtWAJMznDOdchKyvStASpaQLxjtmfuPLQFWleushgQIypNCohNXsGwOCvMDtBOEurcIcUKvWPYaaLkkDQFHdBrzahjNICMueXkGEPBHeJYVBKAYDjahAbAwkVnjlLcLLZicHxpGxlGYTssTPMcCAVzjOTrHchpbowXOQCZDotsUSpUmCBOrPdxtifzehRHpySxdbhInOiDMsxHDLVOJYKogWPEXjTanXIFpPOYbtRakKWyGIEvoFhtHoztVOAfHngvvZSaoRekgAsNGMOhHlgRcOANxdQQGWKpYdgPBMjQocAeWoyeKJnfSQZXJLtnCNRSiCpPEFNLYNCjenmTvjmsJucHoOWAfpgwiKHtrVvzshrNFMtNujyxzFrUsAkZjGBcyTycMopNISotRvImtzTDmavyttAkdiABRdslfBMTrIpLmdreOCXzbNwadhSAnBNbOSGlxrIelheWDwdSRzVFRMxanJyZsiRFwvihsZoJVdlnhPTnHbohNjACtHLbEgKUEpYGpRFTtwGvTgAADbLefgKyVtZPomKfYWShRSTBOxqaKkEBXogCtQdDXtfzqZEFfYGpZAToPAwBNRfMHuAvreYjBfRlJyDjFECijjVPyDmRKttQBmhHCwyBvJVImTOaQVzwzVYUdUakVlwUJMTZWyxbrOksqYMlotSgJjzMQkqGodTalJwIYBqZiuUAULNeZwENGMqTJzUWICdReErWpCYnuKgreeTWyYJhePMMwdwPEdCSefjoFaksOQILUDLjxaIilePwlWkZPWWeUbHEzLazQgieOvhCPPrhFyFJoizFOQfDgFdXlbDucluVLmSPvebbokQRWccqopWEZjBZSMxvfpmBaRIlYOzGuxoSgpoUvGgDlTbzOKqBgxmQCfYqfjcPSiAGSoZpnSujfFXZOaZfrKXKlucVBBrqFRarQogEOGQQEpAEbFWykTYfacAGbWbcAmywiFkgMvFIhIxCRgDNoUGEllXkNHlVAYdjNTAEOpfjClcJPtIsFdVmyEeHvqGmKeOaQDcfgIyhJXfgnpVAaDsscjbTAGUxadUnIttWjshHBOAnlvEYYALzJNNPYkeFnfTfTcZZFSbkcGbTUrfSZwWZvJFlEvKTPgXLViXIfyAjisGJxsHMPRFSNbzwXRAYVKztfYTFpOMReAQYdJFnLgITFeltaMgifVlnEUTDvxZyumsSUqWAKMapQxqeTABFntEylLtPnTSotEovIIWXthboQXyEIfaQVjDyaEzmBhTMooKjhgokOyEzmYRVxoTdwViuOMPtxVkMLBvUXKnHRbbrscOqUVbiOHlvxNwjYttXGuajhzvhySViXDRJOpvhlnEqbjAFUCabNemmpeyRvKvZqffFNpwpasNnEakjwfsKHHSlhPhGEAWhhwVyZfFqJThbQdGZfSqHVksbRmZjwEjYhQwlFytbwsILuNeQEahisUBrHVAhDbCoLSAHSWpTcyvbZxdmDPavWelEFXjtVYpprsIdRosvYuAGdsobdHPXLqpvPpcBTrdaWpFvSlRtswPiacUOYhAYVxfelLoNXfjINuXQhLJUwEIqLMlRMiAMuBZwOFgoUNypJVueaatNGCIZfRsuwoAdtXHXobvfKQRmHKuLsOeIrJmUUitGfSNxsRRUQcxHBdRNAnJYMudHAciphlpLsiwNKOIZXbbocGjQoUMtgAPGJHnxnqUqMHzQqiIdqjNgjeYJssxTTjNzEQeQybLTpTxEgJiCFMOkPgjrtJXznAmhmOTxEKKFhcaQGaQNqBcWqsFXkeAkYUMiCQWeeMdIXTyvCvDDKGFsqeqefrpEfZYliEONSWroAnmNLKNDWgsFkBihytTtNzbnbacHwpoQlZbKhbPHvnVCsaZKmfmEIcoFCdXwCbCfYjwczqXteDOOKhFwpsQkgdhjMArBlasGNNHmIyVNohDQzuGnFnXaOSGzlCZUikUNLCEzAIqSWXRHGXhTQWXndGGidAJLPplNZoPZGbPJIUbMzTryRYRIaoiECwZAFIhtvBdDmOgshoPSRSpYsdNuJcHYMgJwoXTfKPMATxKOsOcpsPEiGSSwlBdsyIJErabCiAVVpkCxcTcBKvhcTQGQsOvprqEknnCmidCEKTiCaByONoOAqswqNHqpCbeYNcUyhbrMYkTRsDyggmBpvDqXPDpfhmpTOOhcJAAskSniZMSLvtSGzIOyDyoMikmghxPGDasbxLmEgfoVUaBNhkUjCyWmJJcsuPAkEBGPfGLQmGqRIptGeBHuNwxXMCfuqrNTtDdtAcjkaoqocfAlmfQVaCnzMLlpuoPRwIaVdqLMgTTFfbADAlFluOmKaIHpkbIqqwfjQRCPZpAFindjMIrEUBqePDotZNZnZAOaoUflihNxQNOShfigerSbENAbkeIEybLUiVEcngTCtHZJhfvmXQMoWXWuLVpKUArxBJuZMnStGvhvGYekVjMkTPnOaEwwOrSfBwNzXsFWoCIBpqIyGnOgseKgBtHmYGtkrJmrPVRnYgAPThoZmCEUpGVfzELFAYVVapDbNLoEpCzKKlbKxaiPmePbTAXWuxUOZgrSedGFkDcOXBddyMSuJITJgWXFPiTWUZlPenBzGiWjLXkIKEQZVjtqOvsyCIzVQBAQYcHwRDbUQFVRuNfdnGTVMAHmWwCmHoLUxRWMMRskdPbERlAUbBryXOotYOUgDfshGpzxymTRUHkNBUDUJzqagBbjYxJvFQNOErBitADadNBCzeDXQbvQFqoqkQthdnFnZXjfKdTktcNSksFQuLrbzaMGTXcOxKJFENZCzDWoZcRcCpTtyyztiNmMWLREugxWrztUVrveKxlBWNOTraugsssfhagMrqfRLnFVDTFReQGiWvYPbwlcBmESMdpVDxFzswTTiOATsWNgkgMoxttidmzNMGRfSjhtcuuVLIxfXVfXuPDMFVRFqzqAqFLqwDpWvSAducgYIZFjmVssVuiqLNGkucplMydQftpXQNPLutOakedhRXuhmcjrkMUcWUKFnfYwItTtWadUWWsDbFzQwOHqzjFfMLfZRjiNtYkceaexguFFDHEDuDfXYPLJduBSGFSpNYymzyxYDwZXRyNQGHqdHZKNlaFraaJregZUyHPguuWaaZqRNcEBRVqngmBhwZLzjulCTZfAjDAxJpnlxQetRMMPRngeggXXsAmfrcimtyuNpOzgGKQfgBxcgboBXxBjcIfxdHCfcMADQlUVBugHVNLPNUSeJARKGewepVXpclJbOhOyXBLCqUGtpuBYiIymgbnUxtYUHaJEITfSowBigYYxhMSLFNMIvPmReWleTHbSntCEgLzFrTZacellCCqowxLvXXNPXSZgkajbGJNQjrvkiQVxMWGXZTaDOqsTfwvnQhZxofYxTLxrtopkzLRgqdmMTGFSgvaBOXHhHprNkNPGANqkdtabyWAXtuwcPbZlUqpCovdfLLvLxOjyJuuSuZMMfmPVqqlJmvggNaxTXdeAsJHFGYKoJDnBmavzDQNtbbHVVIuRPKQZEvSRypKeZHkYypRtoWbvBHPgRPnoADVRwRlGSpsGgeqdtpOuWTUhWarbpJuZjhnuCydWANwmpwRZZpGAcjsQXoHJAqzomgrmDYduTWoTLTKKGVYyeMpNRiDietdunazAdhwbDGdXTJwavHVVRYnajPCoVcqNrPwsiFuMLjIYUEsbDpFFXAXuiSVgHXvHovERJlasklbLNUjKdVhEeFeupcrMHuTmlfHhsvsCvPYxeuoiKVhwLuPklJhlqlUFbUQKEEEdOxNajWTEdFyObaqBqazeVGreGhNJmrQHPPRoYrHraKOETuPjJtoTKbkVByMRhfHGpMSpewkEApDoGOWiZNlqDjGBFRQTOhuBzMNmlvBxlzTBXqsEhIQhNLzqCFnPYIblpXeaFqZyMJZJPStFjDuhTOWikOcPvCPaBeKZQRRYXUYWmeSiSFdxEDSZmblNuKbePRrRcpuagGDdgzaxGIdsoefnGlPmOPtxeVTgAywTNLrzJzWjRYnusfoKNPTYUVwMnIcmpnCHspAEzxiervZKXSBPOLkFzWvFmpskAcZAryHUZYnLwexhLrqMZnKUvhJFGnWzIqEqxRhTCeXQMFKjetQsCZVIKdApUBppUsMIvQzEnXEjpdKGYAkgIYcdVdObwybNmEWxtXZRAeCpjzfnmyDtOHobkmeqSpvMmpBBfnPDsofYKoPUCDnjCkfTRqqrxoJRVbMpLvVifOVcJhBhdenqiqvHpKwUejzEDIiUptvsPtCiMNriaDAbEmdNhlPFaIjIrHTYrpUBMhIzbJjLZzDNeGlNRaHfhNFzcCEVFAKtoUnFJNgECyqvcPpRONBpOJIpFRArGKVGyVOSBlorNXwKuOYRFrNZWUVqgXURCHWzYQCKrsZoIkjCPedlJUDHZdhCPQPmtBEhYJMSyrjQQLvvDAhBVwULFLssDLdRlOMeHroWjMcVmqAgjOmWChhGqPnkmonjJIwhnRjiZqnLbAxljiGrIioFpoAlmENrzblDNRxxtCFVCKwwBJClJEzXVIEffJJZaZUAGbVavCbvIAMjtEDCouQnBNazQHpqqrdBJKTRzkvPLnbogHAbbcmYZICWjtNGyfWfQNYTPfdtUJgVMHHjGCRnwPDgPTpucebXBCJxKeopWLhCmUZAtwMrWOyIEjHjOXDigDlmzQKGkYpBTZwvmAbixZIdpqWhZBqQiYJAQivtlZYbfFKiVFKlgPRLMruwywPcirlQqNGMAeHtxhOOcNCrlDTuBVSwlIqTQOmnuIBUPDKYJNAtdkvhpQfYzTgPnSXqAIsfaMQNpeRkHcdYhjZUpFYJXKYmjtSQzVGxsdECRCsFdidjggpvUuTQOCLLgVzlFvNDUDDizlCRySKJVCcWRzALQKfxLGQneSpJHWrADNzmVCAZHxExoOYZuBwCygPxLrZtOQogiuafOVfNpxRZcTxsbwhGzOzSchQGAUrvAhffhTXzHadSLZniFZGdRtlQTIFwvbgGHBIgLntJDgHXIdnAyqUQUNDuORWADHNGaEtvyeetFaWKyuGLKbySwGEpLLrYEIKGJqtHSrjZawggXUvQMxQErYuvhFSDTkJqXLNhtByYOnPVIHiRjdFqpBltOCFPvngXODIIwPSuJEtZFJZLiCHUmxdQEmDbcuxJCYWIAustubZDPwIpbUxiWILDVCGkbCQAaaocWssIjODDLctaoyycyLuuSPvpdHsSQeiFPdpNfcpIryHsZfHjDLQlheXtWyLuFMmurQFHgUoXZkXLyjQbeSMRqWgcxtvOXBDeRYIacUjIfXDzfUyGIKuDCQRxQFKdWEEgoDULneYiAXyegFpIrtjDKxKpWBLVKwSlJbHvzHJazjBKdkVizYbkUdReHwnejHRSWYPDtOYWpabETPdkJcGAqgqqOpYWrrlUBHenpztxWGpqyUZWERdKuotffgYUVqgjRNkphmanWKUJJFeacuEUWSbVRqJAFZJtYBWvSuUAOeaFdKOoJvWrflTAgJtydcxYlCPwpDlEmdSWuWHhJayNGGdflOpZofmsDxVOIUERyGYdTwEnySNdfmd</t>
   </si>
   <si>
     <t>2026-09-06</t>
@@ -305,16 +299,16 @@
     <t>2026-09-07</t>
   </si>
   <si>
-    <t>23:25:36</t>
-  </si>
-  <si>
-    <t>23:25:37</t>
-  </si>
-  <si>
-    <t>2026-09-06 23:25:37</t>
-  </si>
-  <si>
-    <t>2026-09-07 23:25:37</t>
+    <t>23:42:29</t>
+  </si>
+  <si>
+    <t>23:42:30</t>
+  </si>
+  <si>
+    <t>2026-09-06 23:42:30</t>
+  </si>
+  <si>
+    <t>2026-09-07 23:42:30</t>
   </si>
   <si>
     <t>{"key":"value1"}</t>
@@ -329,40 +323,40 @@
     <t>&lt;root&gt;&lt;key&gt;value0&lt;/key&gt;&lt;/root&gt;</t>
   </si>
   <si>
-    <t>Dj</t>
-  </si>
-  <si>
-    <t>Tb</t>
-  </si>
-  <si>
-    <t>Jq</t>
-  </si>
-  <si>
-    <t>SGveqFGoGCENYODnfOllJJhPidMXREXVJtRfFpcggxvoAJrxKlFevTtxLCsVSzPjrQakeoVSegjhFWjZTOdLoWQuIQofAxRaCpIDUbwvQTwIFVNlktMvTOcteSWhcgDNTERPJMhYJNpjUWALFVEgLdwfSHZhHactTDamaEzZQjAwMKsqFKDqKrpcJmJmPaFMtbeoAhgSYwVteTFVxcWaY</t>
-  </si>
-  <si>
-    <t>lrMsVGzoZOFWjCIxBDxhgrDcaBUEJyGeRJSLbVuspqYIpGjkFTOhBrYebuQHHgaPmzTRWyvleXwtCnnEymAeUWgBNPHmpvnawZKrgTETlCixJEft</t>
-  </si>
-  <si>
-    <t>KsoDhPXzmfSBbfMcsc</t>
-  </si>
-  <si>
-    <t>fGfEiLbfSALAlQYaDRKXHMAEkhleYJZLuniAmvJZJWTAQvyVJnlzgjRTEBoNBOxrOBHrUggllDvYtOTVHAlXNLREqRGYpaeuDSOXsUpntfkWVBboCdQjXSIJeqxCyoJOAvFJTVNbcAQecWmsIysmOJmJGahSGVnKfdlQOxegpdgIidCpkfZfqoqybReYiYQHAnpojDaxJpidUKupkXFybmXGiTFLkRmBjsAQdNcGQOspUclLFsqmgrrtvoRwXPEAwGXuYbzmkFMqDGMOmmJKQLEqprkDybqVENQjaqvtocLhvIaWgDylFfgvmhYvGVmLykjENfxwrOcXCtVaMcaHSSbuKkjgImdOhQbsDjhxptIkcWNQCRogqBLpwACxcwAQwgzJOYxvzHyoPbQTWATBbyBvCiDttqWaNVtDnNgFgUBshqpcFDzCRdVBLrGGrJGnJHahVbNaAGaCtumHUNQwrAtAeoHVCjHSvFXaEaXAYFWiWlPxHLieiQVAVqGaEdwTpALpxJylsHnKQfhjUWUFLZSoKGHpFcXJdbYukQSLrxBbeRDNiWXMuWNWZTkGqzrZqnqZYFLVkyzzQurxNUPNxTyupCMURchsIAzhAxHfHrJhJDbvOEQsSnolCCsajgDkbIrHaRtXIHaxLyDzfXqMliyCxZWNJeQjOGdLEVEJcKNhWxMQbwhUbLGrFPGAjblPGdnPJrjNEKzBIpUiBbtaXHvEZdUcvtqajryIkjnIelWwGGpKFnqJhHhqvGezztDgeBGfZHHzcYIPcAgoBcYYQYuaWmduhFoBuwLcjuXkaVerjLNerkpglXlNedRlKoKJLZDQjIqfBAtmszsOcBlhiamvGuvlYEzHiniUnhMDPfUnUhAfhibPbLVqjPwzJaTzfAwsualEDAPrcHSrQhDIHVTfbJyWleXJroQFCvBTmCmkmxiJolTpkVsvVYrJbziSJWTdlgzrjJSHqQDjhIJYslsdIgMgjGapakcOaGHDuhQmwUbYuoneRKthxYqpwTETIZHDsaoabOGJNrblEanAFYNpgIhMuxDMFebssGxUWlOSrwenQAVYOrxuxIlBLgZJtWzXySfLCjzWIkaVhWkiuNsuhIUpBuvxiDCRkDSNTVzcgfoGVCeeUBBOOXMYCdupfqwEcuuWhtbFETvYbZsnTMosFnOSfcgCJWefmTFSgZsNLzDxZTTPLViSSPCJFjapqrsdkhIFmmmFEAlVICoCHtCIsDKrPnAlEdnaiXfKzRIYXgoZWattkAQHbWTbzxpyDXObmNVHLsmHZSuxOOMKDTUtLbCdkRVJbMnmDeHulZxeKzFIGNgGIAxTIeFuThfupRDBPtzzpIWoYJTuwqMrzRvTrQjsStIsIJPZYIiExnvUgNxEHgKQZytoMCBkZGQZARpPcEnJqIGEKvvvRThqotWrTESTmHYHVIUmfZJSyaTWUHYdTrnoUHjUnCqUnMOKBfDCNIrZyOhVegpBhIFodHcaujAFttxuBUAeQzyQTqzRTskxQLSGOImfdTgLWeZCjUDbMwohKiCKJTNVKaCTNDHSpLAPhvIrYbHHrPWazmrzTEyxpcQAviiRSYuDJXELqGhLXRqHaeozCKqoHXXcAzaWuDfpdtSUMSjrquPDfFWZxXWfkogHhUdqQAuvFaBmLDBevfzAPVhXnEAKUZvXCSZyDSRxGGSAqvsAiZJmcQkWclIsLgvilcaQHnajYgkvfySDOzFJhSsnncxVknkXBHsaDVaMRsxweuJOfltBdjWuEGdqXqWARcwQPrlhXiQCHLjxXaQlkWcHJAvGXZUmzdYMGvvXwUuoQTXOklSsgFnkrYjagVrEcYMAILRKufIVWMERxueqJYDWlnVPdtQEBMpqkDHOYWAJftEWJRQGbQJveOxciXMnOjWVfjODakJhFDnVfEZmiENqEfqWVtcWStzVsnGdzUVDYKBBkjpunzDVaDKLCbNQqcnFyhdTFehAviLDjyhUgRAPMOBfVgADzvKjuuICBAITuRNvmXWteQvykpMBLCzaHWmRlzEtPqxuIUMfAYFezFRCgLJLZkhBFIAANUqtBQbcSqpgLWuKxTvNrQZHSEHnxdehOzifsDXcenicogCrWXOXOtVICfeuATGOubBnTeKmOpDDRQpwiOUDTblsBIkljvoRsAtKoFpEieMBTZmexAhJrHkEClJWNkkFLTOpXGXcTApSoTnUazZocLVRGctqWYixucPmzxnBKnyAhLCabNmVXKtnAYdgVclyUJZGWcCqDewVlwqweqnfMGUqlIEjDVguZzbVUvwqOtDVVpcWsJVMNvhNnjqZHuImKFgJDeFvopgPBaSUDFxBNLTHAWFrEAMBAIwRWdzclvUPteUAMbBBPVyzlyqihcuMAFIlcFjdiWLBSxwqEtthjtJiBwsqpfuFhudIUlwrdXiyijrmchijzvnzqBEGxNgoNZQuTceklOIszYlCPmaEfkKbdvxSyYuVSjWHJttGVUTJcSOwAkpxFRSpqHOyVWogGDfvAYbfZrMzOvZTHvRSOMdWKrAWWvOymdIKbMGxutTVtkpmvvBzkLDdqThibYywiUeJbirDaMbZKrYZDwTivrfvinlhbekNKAeJupMSesqXKQkeKEpoBWjTRfkgJEDrYzNxQlAUPqOkkfTtoWyZuSwhPzFBwBjMIygqrafFTuNfyKVVAKZYkesdTbyYyKJeRtDSQzqRQywzoXWfstEYjsiIppPPoQleDnGJMboILeynCaZnEZhXpfMKwdvrUVrjjKSFhXWdafgWwlKBFnrdUwFpVyLhiYyozFBwBbgFWipQIidCSgMkThOhYFsqJOMASVpDLDsjGKaCinrizFSvVopeLryEezEzEYMHVaCvYKKHVoDORckdZTjukfyRNCwihKgVEtkbjizBREpzecHSPBrYlAIyRtQZmrkGSgTLIQPhkiFJTiWRiDVQQcbdYzGGniUkzZqHOlFodJbpCpVvdVYEqZegBYyVPLNXDpCHFFuEIMzACRLiShYvFqRQWvthWfdZkvYiMNfObLPwBSgtDAYfyuaZKAbrOrPGWBnWbEvaJljDCwFfpiFTcnfgtIDKmULvRrmbNkDGpBJNIqpJSVtFestNaltcrCzURtVBLNtVcpGdyotiAOIuANftxGYtLxEwlVblEsizRDQyuIAolZmSddpbsvnesnPykSEkePAiHFizCIZjpamwlBfhUITqYBciegnVbhbXDwocZoCOfSwUxfMkJlxaKNGEjGJeYuPXTQyPBxzMVdKWEJdyKcAPnTphxxrmtLKxuMyESvIJaCsFsvNMbNKXzgdcCndXgEIYqCRXaIklxeULCzpCPevuqtdntERrrmvrjKihMFKazOmBQxPXfWIwAqakeuDyOXjUXzYlmthxxMKjQUezUSANxVequlROUoBaVqhjQLKaZxTypFeDmGYoLSLEsjmFVfzfCWueVJzWYzpZTYmvECQSXyKKGELSQQIcPUdIcOpiXZJtYdOGPjhSVvkHPnCMwvEeQROccyncvqHmdsPVSbwfRyjTEcRjRtdNwoeRvwKOnbUhbNueJFtdjZpuWjQVfHHcSyQfxADXEIPzOWOUAURNskaUOBbnRiliPbEcTyFUvanKbbfScpJvgKCSXWfUCLMEShpthxQNYSFntszhoXaFYalmHwOGrFDXYikbsufwdDkmLbMLvPKfAIMywHIVfxOoJxxGMPTXQzqXUAflrBuPIWLurIPLGqCAcjKgEFTuElDLOjvJohLrnNdibsJJNxrhFIMZjIptVlNBuQrsfjYEpcGbtdiVrjvQtcaVCyMYbHEiNMHVXrLbPXmfaOzMzDgHdvOgqFbIqjJPUmgSeaxrCHSAUPCRoHeqVQpsqratTjnwKkWqVIhFTONghrqWlTQfmhQRLirXefmgzEMsTfHCaCgJEebnHuMsEXyCXgkvFGiLNRuspzTAqvwcEdQnVQZQpMZXSDoPWWLdoxGptyPLDMTiCrYIDUWFfkYAyotkiUwhcNpPsaoCSVymVHCRQceFNKAWvQxJVfmpjimeYLdIYkpSJAnVNwcyStmofMPBFYgeXxkuANHkiQRGObojtOLUgSQMhDgPZXqsSrFWCahDmALNmdQSOtBAYSacHKuVbzyodjYbEdLFhAwQqHdRVDcPEofBtBRwJxeadGCZcScCqutSuZwrwKBfsAxvIUVjEVObrYMQFDmarANcPawYnWUGHbyBGhhDgkMQVsdbfuaNmvUiwkMaFGTsTTlVarOZxBveDCmynXqrUKhnkcypiiDhYJwqMeLAUDfFuQXXPAOUerPkkTWPLTidyaMSdzKHxinTlMKJzhGdDwxBZmtMtQkRKXzZrxjhzBYePUbOtlaeDNmroPJqtQCPCKoaUNiznhUPfnIpztXQBTnVpQAWhWsURfNPZKstdMsTIVAktZPbjZGRRyfzhIPreZAltfDCCuFXJTVAHTOCjwRRrAVAQSDWFbXeTQZrXfGWYtwKJhrLUveHJunhtpdvhBdoSQVJtDYTlGzlqYtpQNlusyyfbCyPGnazhpUcBvtLwIjMNamEfEcuQDEtZGjHIlQDYixQOskZjRYxZjYDlpkRcMyMkprfGbpcFFzVYwmCRcwmNbLBSWqmWaKVYLMyIlpoJuUJrJImUlRwgHupBeooBNIeNztnubtAoYhgEFtgJYuiEJgoxCtrajAZZPlvdyutfQfoJzicmNzCORkkyoucGXLZOmitsgTBBuRCNrYoOOpdSsCefzReMtAFteWVYvOcrmEhSigIPqkSufLVkOzRilkbVXLOlarIoLpLVZLtCyPZKmjGwEbptWpHyjBRBGCGJgGJXGBKowcCMgnRkbYWtpzEdmwiShTSDSKkWYNkTFRwCUWgIssDdTAvVaGqnRBBLYATciDsNwhxtiDgurdXTLPFyYvUpHCytIwRfSrOkQuPrOnJMibhNkVKjPpnVPUUwdHeejFSEIKBpLxgcNVzxQviDPxIJJPZkEPdRRCJsZDgQyMWFtIeXNEvwEbEAGoGwtOXUNuJmFoOuVOdmRoUEmsHGbjBajIiSCPsEJIorfSddJYeWReVjbkBXsKgRWJDawnlAVnWqxrZYsXbDkbEovsXadjVPRLQflxRXXgbycANGpssOIItrQpVYEholJAVSsafthusGlToJhGXNXKIOtsRSLImWbDQAQuEqRZzuhZjEMYChgRXHWcXCSMhAZQjOYqyaOLSmVfkjxTfjyOLrytlJgqzfYOIQxFLVaAMtvceEWLWpmrjZtxkFlBSbCygjLfKvlACzRTTtWIqGHShxoIQjmicrgXjntipNzWxOQpjoJbyfDCviRasSJneVtKqEQwTfmbXDLpSBUXdcgYeYsomFrgsKXoDywFtINuHxWuxnFFITFBKVakCnXUYdNriKaEpgLuWfsKthdTxYpUKIcaQPoYLubNcaYUhaRsiGRMsgATZrXcgjNFvQletQftZuiCoPsdbSCTIcRISBvjOSbsYmueVzNTRZkFkNgjxKHGEchRFnMBLrTSLOeBxswiqkpBIcpULLTSbBvzMtOCWMvPCsRgMycyAwvKhPoiwJeuSqHJDTWPmrDNBmCmaAyBOnmqqaXHHfuZsLgzLnBSMDyaUYRZZeQeeIYVNQhbVpUbJTRHbwQaliflhxyiOLRLiznZvXGUJCLbQAgjnWPOHAEGjjTQtAlgAmmWyFNtkjZRfrtvFGXtZVYgwRqNUXUeBRtRnCRRNMaCfzpneNYncnrVwFqTPULViWNWukuLIyVCzzrCXVOkuPIVZXnryYqKaoyJxtdtZiaJDWtcznrmuihrlYujgyqKMkOYFKlhHRQeqFDKmMcBhpgYGXcPHUdUYCNohEMDARzTcPZrOCIZrMjCxUUYbqokMTGHijnYlneBOniFhLtYZeGMHTbweAFpvKaJcQNpYehOXqHLwUSCpmyGSibiHeVWpUWhtBMJiChBHbpOqluscJEPjrLrWEMqesQfBKsTSGJxveRmWmfduUTabZBTBHZDEawrOknQbDKdwndUuazJdgaBnIeClXcaVeknGZYkNJBHRZKMcigVZSOhoYddbIznLNCfrrShXWgIEoMoKtYvCGEiRdzPisbljmZwjbRUiNYZLTFKQEpNJRLyhNajqkCbXlmnoDhWeUFjhmiIAuKaDxeiaBpTLwXlKsEEVGIYMAChfuuiFGkWFCGORZaapgMpzFSlOhQBTmAmyVZAQzTLUDMINLKLhXnbQEOzIZWUeqflVNsNDojLgOFymZSqMkShQExjOaACSfnnMhgdCFZoEjEuUyuwwyJgydnauHSvDBdlGRrOtDhtbsoLPPmHDOBvuBhkHFpAiQyVnsEYGLacCDZNQLMcaQucleZLyCYrGDRlZDSMmOuGOiDIsGbKDzZiLEdriXLLmKczXkqryyOtnrLZrSsivjGOptwIHAbPclrKjnEsVHzrenmGWOopYbGalQMgDCjiSQVHuWKrluyTWXeopnUvklZYdOvapjdxUyGyAGBtCszdnvwcGOLLtJSWLVZvMbAyMorkBbCkRObshmppuekHkjHENOKcAJclzfxHEpOtStbXrMETPOJJgcJDErKJiyrUqoQTOEJvdmuXCJRIPaQdLegtjCsUQwkSQTWlPyTHKLeCsdhBywbLUxYQqmrppDgZfUQbXoJvvpcvTIDPTtvzndazXyYmJxevOmGaSdQRkEEuUjsmYHJmmItUafkjFsdAJUShBCjHQuqkXnJdKasYTbdRIRXJfIOidotwdRksQGEtTneEyuNZjxVbotXxGdbJknbBCRPsCfjIPVxWowTGRlWxsGeoSHSqtfqjBJJdBZPbMyUKzBzfEXyhyRqmbKqOkoxvmJDmkdhPeajrTyeWOqVMiMlCRqTSPRyZhtqQkdtkuNSkvZPAUvTnanqXHQUIizDTIsAACXlYeQTArgpcQDxEvMKwZfcHzlptFpGbaVWliyMRiSbhZTRWwJJQJqtPuvNoYNxTajmYSSfvdfynTbTjwwrvaVbQBAjmsBuLqyCHGKpjaVIyeAdSyvgyDmEgroHrVTukKJLBvfrhUgoRrEnBtZacZvfHsUoKWtZnfuPMDuXhUOsIBvGffQwCFCDdeMikCvjjAotwCUQJZRKgpjfRDAHRELiWNLmMBcTuZLiKkBNQQIWiefSoVAuWucgVzzYrYHHmLFLagnHbVXzrtmzLRBMDparfcysFftPYEmfVPaoXpORDLvyrBXfUTxrFAGSmEylWoZTMfQRDrUBessxuFkjhhdHBsvvfyZnmSKDlTADaAkjETnXIUXPVZtaENIWdIJqSldXrfNnxLwoSrXUkzrONwnTWanjfRbRjdLoANQFSNqPReqOjxasdioGYkiVclplKWpCoWlUdYPKacIzmdBWejmFNVbPLlfAVhJrKYRHIhXBsqvstWHlNHfdFzvZEeMKdRPRJCoYseiEpJktHpyuMqOWzFiwylOiEsXjbEQUXnMXhecIOJTKPMDzjGkSHXixUWbTAgcVHpymLfThKIJgkNBYBbhjQgRSHwuCwbMZAbIaCYyftiBQWukBGggdOiXHLoedvJweSCnYttRdOOmOSEFIHlGPtzjNfNeTwnFXnIHiOrmdHoDufAowBOHkxXERVkacwxUnsaXmpdZJnhwIhYaUhbiyYLlyWiHjNlDWdjKUOeTCRWiowepWionUMvRzuHCKFdGOBhHzpYpLVeKskoUQxzJpsotCyjyeBjkNSMUApttnkbDzlzmJltXVbNOgGXGXMkOdEzttwnYMXEYGSaKHEMDdCHDVhxkQZuvXJcIesgzqappRtoYQhfPwBmMzbvLUtczWVuXgihucdxqXotjdHHhcoywttgYqRTpmKQqCcXWDwBmQHkZHNUInFMhvZZCldiMuWmWwdvAUOywzgwlnZJdSmGlpFsNzjWYNIExFqWHtEzOlJUvBFyoDrepTNVOcuqOWRyJUveQZleoevetNPnbpOlkaKXOaKQVnKeFSrHkiTsQhsJEeCuQAsvxhGkYBiCqTZYxuEczqRtOEobzmqjuOTVvhsfQILUTaPYrukAiOiqlYewvhwHimXSNVQOKhWBmVuJnxDrQIoDPurgHDkQcRrgYcZXugLTpgUDZsszOiZCTwifTOUhzstpyxsSCvPofDbbjYJFIModEumldQiLJMfyHNqmyZOFNSagSjifayUTQExIIHIRldqDOzntJeGhEYVDxxrXEAatWUUAAGcYrCQLMKCEaaYzsuoxundsBtZkkApCPQQKaisbUEXBAJMGnOSQNXeyWjkVnPBaQBcRFczgtRNnTcgOiczmhgifzjHdVQpEcRudcwWmvbVvHBOtzsYlbmZQjWikrmpiOvXkNFgvIiXIGVrjTcIXKJXnieuwjVORyxXGBpAoghfwttJfFgErrxCmtZXntJLRudOWzhFhnLlNyTOflzsrzjwQjpAszPvuABHpyiLFHjDtpileQjpWnXtHeDxfUBpyDAcdjfrDuFoCMbUqgWxtbvlnZTIzCgSflEDcVaePSBprQteOBJRZAHipvShocMyBBrDYLffCquKTkJLLYirpmCauQvhvwJXSWeNkRXrVGUtQHDCpzJYnMpIYkBfTucMZMhXtdAUReMwQpWzAJJOURwDIXsbyvgDRpKlBqLJYfwmOaUtswYmekFMjKQgdBgBWGuQoxXcXznlPwtSPikBllEubuqWSLfhzuVkabxdHYoQPLjCbjMRyVWsdtEkkivNPDjEDblklOHuDNCOLpsvLpTUKUzPaxqGgAlGmXfauJLeubiKBxrSjdCwtqaSXyvKMARTcPwhVwamhBEjAArQAGipKCsSilNHeYJssdtMXdNNfghsAyxUikXITGmEwmExreaowPvSGWBadPCiIxEZWwbfWFaiLLUEENIiKYGVWIYqRQUFHdVXUglHvppCzbdSqeQTPKIRbOObEJMsGFjZnRPpzFCVIKtTRzhoaxAhSGEEYrFbdgaeKvAViXnKEeCjosTLErvgdeAGARsNlKxLlyYmGCnJuqbiuYEMeuozHAJmyrnJGvjHIaxzrgPXygSOgFiSXJqkCFTmFlppoWeRcnqKodsiesuwUGWhfypRYeNleAOYTIWXIZcjPuBMGiSlAuAudUqTQbzgTjkLKanxIqzoxQICApEjGGfsJjDgatfUqARqLIenXlGikidCXwdiVebAbPfdRwvcfrzdObqmDvSgpfuxWixvqxMPNTtByULzYAUqgWXiPDqqrmbkQxoIlMuYGehWgkjsKktUXSJSrvToSTunQdrcKVNvAvJEOUeZnqVUMLAOrXizJtSiLRerUrUYiYYljtfofMMINIsighQXRrdDZCGOUibUqtOXSwPwvVqbzgFruRzRnliDdZqmPBzKceWlrzZhYllYPHtKKXhwiZbmgmYiiaYnapGkutsgoTVwAKWDGsWfmgZIOkQjogipHwItGJMKQBVRCyXRUReYnDSLvWtsvUGZwCoPrEFmJYbegGfshCXMCJifyawkWwupsbLFtAnendcUVUrCJflpJUyooBnSXreFGthrUMCRGTnrLCpswPoWcyqwTfCEjkcxEWvWMXcNcGUTBspFZvRXZtqGAYbHNAWUWrdmHNDLvHVRqVKHFapeoVVKOdHYOvsSSUtGbTglDeFiqujhKZoDSdesSyGWBHZNKBWPIQUvSBYhSeDkQCLJutoRWzQAeXecjJAvrvaSQxiloWNNwOmySymRGzxwjyupGABBUxMmBgyCIbYEzeECfuDpjRMRevdHjRMVhabuMdxfEMBTcEBjvRhvuruekYUyxekShykMfNsBHPfVFZukrUInapFZnYZKTFbSXRXLphqDjWPWVHhSCdNeaegCqlXAOqSoCXiDBriONwMyYYgShoYeFdAtwMjeDDGtvwyxyFyxNLKerQuzDoqMMavuDLppVBEuETGVNQYQrxgWGyPYgVDohTIXOjNtJGUmotPvNwPDyBsRfVwRiyOqccEWseApwkRgLHnZZTjTsooyVhBMDLHdrhvMOUcUoqCoAewmSlrrzFLHKeseeOzAifoiNbcbtNPMadUNPJeLZVDwDcZMTplxjIQlhhbKIBunxEiGjxUGOBdeKvUtRyWTuvGKzOhSoSdoKoHijkJlSkqriGXjItXSjXCxUhCZRQSyyPoeSxBRCdMDyiKjnEPYuWhHESLORVoyhfzgESKIkOGNIJiPaOtLIwuurUgkczlVCtMcEyBTDCxDkaoKpXuPfZPKPTwyjIZsWmMoHhQwcYZAxihIxEMWVEzhNlLxXDIOpnogbOGcdBchePIpqxQpNiBXdZrXXPnOKFyQedpRRPYwKquiJjFTOlpfJPXRyTMaUPlPjIaAoDdgfiuGImUMDmVzsJzOXyRwBFSmVbeFAsEmVbRnZwEvcyhXDBtmDqtJOrfgOHsenaGTYYMlUoQIApzaGDSmNXLSmnYiKTHhmeBGRHNkTHGCwqAccqKoKDEGFfwyTQRoLliNXwxkRZnWKFUOWjphhwOcApQpmcPlQWzSbnOdoFApNiXqrNYrCPyZjSkoPwHnKOwzIbkbIKsEBicTVaNoaklfPhRDsdsknPflsUtvohzazUXuueqTQMgivdjHgJKAwjjNQcUAlOLxnJPSwrWivqGPXQGpmKrjhOTyKLkqNnqBhMetFtkDbemWidFneQchEJjAAzcXsVDtCbnlROpjtUuQrdhCrZCLtCUFwCJzTxXFyzUDMkPoRPdYVoYpOFnFJODpvObHrMYXaUpRAqVuylnMLAWRLIaoFpFCNoSUhqneVJknmCyijkDukJLNwNUgnYXebxVwxODvbCIsrJhdWgkeceOJELkvxIEWXQIwoSpOhoXpfoVkKnKHQleVKaOkNiUYpDbcrJiOjmxLYutnExufTnNuRJvIiUrCLFRuvvguBtEBHsbFNnBnxXeRrTLftgStFccQiKIDBczwntdFxhQWBAUwKuFCxZUeCXpaTNbGjEzYdfomFtBgwKHHlCsPwObGvTzELyyExRCGEZoiOdsinPIdWAlLRRhNmrHMDEPcNBaLchVKEyXRUasWYCwXULHJGXqroSwaNawBKNwSthUGppLMUlMCdHFbMYnXeixcZjdtKTouDMGlPkYVjlXFwQYKCDGOVbVLVxnTkjQRxmdiLVggYaEmrhKBgsqfBCPozAsjzXhRekleJFsbldnJIjZRolMifYHhyKNfkwUoTKkCCsBobDepeoHZrSunjfuMrJmXwEHVXpRmVuCpHZjCOzjaUqeYtWquzWiKqycDvnJjFyfDYGweaGpiyYtGGQiFlPmqtVidVEnyBmUOknLJanOBiFXVtCExcukIygWgnBdboBxvJzcdDQBZeOaNnLsZtrPxrKdoeWtmtZxODYtyOUQNyVFuqRqVoMKuxFStXJzrzawAmFHzXbzaohPGXGpMngUxxwrNXBiIMLDAdgDkwsqJKCxIQtSQOCwyryICJjCvBpneooGZAdzlEfmfMFPNiqArWyhCNyPOIXICeoXnxaePIZrVRDIVxKdiLvIwsSrntEsMJqvOdnrEbmZzdxtgaTvcChDUWsXEYjyMCZzgNqbhWOONkisECQlToAZdBTiGRWwTVvAOtkNWHZmrbhzbwUghEwHjNwKzgjMdswzTZLlxazfRWDAcMTWkKnaSNPamYIpJZTEbYomjPblnrWdVoGynQEwZGBgAhMtjeqjajxOBzdYDlKVslNaYBeoVkHeEpjtHyBCQZshqwWdbcIsTvHHBEPcdBTAehQTkjVWWqiwDGTiwQoLLqENKCPIkfyMZRfcJYiaCVhOIKvBekIENxjNqGNIucCuNolzwlTlLOqbKiQgeQCJaWnJrSXgKVQHTzwiMWFlEECljkvHByogmbWnahAQgHMetSzjQxmDFUoejoCdrPuSErortRpQETuJZRiTbwqGCyLZWHrRJjpQkMnkikcdPDeaGVoumWymJcGAkkkEOvTikjoLqIwvULffwXYmRjbrtungblWHmtalHnWyPFNkxpIyVxiYkwLPIjFBpZcQgkpUiBHykbXPYEOPtGkNLSQhMoqwUERHKfcfLbxMYFqeBDseAljHpOWhFBsgcHSstzLwemsvldocDydrGZpNrwPJRBahYRUilUYzKKVIKXPWXdsWADgOoeOhQaUmMRvUzVWbLZokYyLiCyVjIZFebpLtfPofetQazzWTAsCYmRZYTpKQDUYxMTyItqDXdcmYyrSZdfXltsPkYeTFqHiCiqNktKCvzKeVAoknYpnifjDmVeBATliKNOExKkqkhBnldwgjiujohOIZCBhKlUFCstguIdlTEHJPhmAAVacrLwYgXpiJbUbaPbkcFoyfcZOEuRCNlVlpMFNuEXXAmzRvmuPQtwxpojjAYdMxePgyKtVtKEHrgNCjbNYOezDEZpZiuUvZllRSNwqyGnqBzEnxskfWxstYLPjqHSznUbZPyvLVxTbMjdfRDUVufrVmAMBOAEBnlgkWzbOMvBhDwMmhGVDrViuTSRCNeNcOznCYPGNzIsfhMYlXpkbXLggAydEwQPGPaBzaMrLlYhAQSzWCNQpKYaJQZgVpYEOwyVJJOTZQqNxLvjLoJSBSobghEWLvxcdWxSsXGhMicDuOsJritWmHbYMdVCXqlaFKPDSiruKTbjcBuqDphadDsEPmiSZWMdwlKJFWXirIUlUbsQVkhRHyrdDirNlLsiOIxJcPtuwVVQTGZzQaPyZrPhfcQgsXsVIYWTSQusWUHQbLvvNkeMUEytvXIftVywVGtlFTkOSDqgtwlVPQKPNbwXxNZbHNFsxXaXMsPnEPWaufYPpzSxmBBnxBTDZgErVggIWXBLSRMPXrNaMBPedzraRhWRaziYiwmSurEznEJOggpvoEWJGrZlcmtmlcxNiwWxXzLWNfDLdTGeynPJaKmdsnHacrDmFUumowtSvQvwGFeEPvaFVZUsRpJAjnVagPNyOkuBagFMakhDjvLZJBLRMyOknvwDORvyXMyAZdhqEyTsfKFLegGLnKJHBPsdDSpBlbTaNLRsXcFBsFqmVFEevzGWdJEnhGSFYFPawEsYgYAKfNCpLsRNIUJpxxuUHcbCCMjYoftXYBxvwSqoOwiCqesJZmkFvyCwSPKtVMJRqAlyppnWTWteegDjDEUWlRVXKMpSppfIvXQXJxpOyKVaiUJYsmWkAIQTWGGSMnTMykakWZczoSQncirupOdpUPszhMYsZTyaOdLPAyvxRovtHjNyGmZhtmbeOWOsbdGiUKzXLauZEnPRuRrDIpfrkwEOuZFLhMqiPeWcCXGqYonDJrJmxbqXfXXrWOAnAcAbYrjEOMyHqmRgVTJamRaspFQhgvmJlzQCxxCIXauWkiSkeBXpMCREsXigixeRCtpuaDyjVaQxsLsdfpguXmgyqyBbAndKYawLpkZnkHjhpjWoXGRdmrdOdNFpnvBszqEKRPuGwYRDpLRufwrUvoHiwlmhRGVTkgCIOFvHtFrPcZJgszmBCLYeNfpqgvQOOtDEQYHopTfVcbHgdJIxdGIXcKTqQovBMZMGNCMqCWUdykYLzSSjKxjaTobGJhTAEAkagcEuwxOTrsAxeFqAeMlwbQdrOXiqvOLUrQXieDTDtzagRWAAVzYKaEhzweCrqWrVohZVqkynaPkHnFsJYSKtTIYhKPqfEoDlifoGjfVpzlvtunbLVKeEQjDuiKNpSuAayVqyrAfrhMhwmEeZMNGuIReKxpXcJORXmHkomKYSdNVLFTVkTqjGZJaSYnKWOuWaYcpLTAHnqcvzuonULwIaAXTaxshwNTbPMYMJyfkivaNlYrXBSxnMYANRJsKCzkicCXRtzXcxaXEyrezArVJaiMHUhSAKuFlQgPPhZgKrBtRZLjjwlWkWYYUvcFeEpWmFWIzdxlftPMFkgIVnSBTxJZIvJvnOoESptEJNYdNUjZAiyybRrAuYOYyoitjbIWVmGVYNuFtdNdWUPBAyrqUEdqJEXubQEybrApnqawdfEAkQKCdxUkwlSwZWPHieDgUVIbHtmWQrLZpnaEnuybAKOZiYUGUyugwvONztWNzFCjLvQgyjzdMnomBFJJgcNCAWJLfMMTkjWCYgmRFLuGcVgtDYUgdmQxLORxfPKHqKVLJGwNSqgHOyYdSfUFqIrUVavSqyxBVCwemHKVGJgNxLQMilhXWFMJzzVoMqgsWLHJqzUVlqkvApMljFbpPdJbSgsLBtnFdXShLlxshiAZfKSpXusbDhrPmJMlbgJLSdEMwsLDxcgBETJWvMRWUxSeOGDdRXVpEWjtjYqBjstBAKYsDmJNQhkZIwwvqGlbIKTQuegMAbobESjsRvtmgJlRgUCMIdMzyUBvvjRYwnSMgLvXztRQsVbsETwYjjxOsVwqXtGnSLvstxCAGDVodYcrQSpYiqhjwsHBPZcXNuHhSBOmGKziuyaJDPLAjSuwAPveApWAzDhqOfERSBZBjdhBXKULnzcRCbyQunrpjUEIvkZaFQLgskCtwlXTuXGOyloxhXSsvoABzUnDihMmaKTmQTOdoeViXHdEUtuNLODvkEyzywQrPvOmqOzjEeXwHgWzIlLeurpnmpIeuPdIJeEDqpQTZbtBwkfRaeEObFkcNlyFDOwItuarNzsrqxUGqHxgcUqirQptaxEwwshnvflUozedmPmOdQAZdxXKzEuaUzTUFUkVKGOJLCmuHtakRtMiqmWKKXcYlllsuyPykgrvClXDoTvxgyLcfFfdlmnzXAVNvKJWORNPiXcUPUZByZLXTCppcpTzMZqHZxHrHrdoFutVNhcYIaGRlUbagQBppAWZuMfuhSDrVhTtmeYWGVWfqvyBrpGSywAYxsnqNGCNoPYzDkXlWZDLSHWLJzFpCNtBCTnqMovXYmTYHlNAhwMplCSvuGsUYBBzkxuGieqKOHfGWoMPRQIvNnUvRTvsfFNfZYKOCZCHnUlJfxEFAfLapzvMRRiPDYIBJoylquUoCamukWrYpXuFlLhwUYcXAWXWMpyHcHTqCHAYdGvyqcdBzGomjvMdhNRfOJdBCKemipmhCFHzFyygCSxpuWhmuICmRgNramItSNelfnLkDJeEIsnYIhlOYdiKFAmjEHBdwRHiLQXsIhrKRWaGoyNMDfeUfuulzxeajPOiPPxSZQJBfvbIRBxNyUFnOXKkWUVfcRYQUddxTzJGZLItsEchwYcsiXcnpcwNtPouYsARHSTLGCniilXQMdHHcpfvnQksdqmTClJzZDcTDHSWkEHjJRbiTJSxsgIxXXUwgRnvptWbDYycMiIcRLXfhgjHdtMjCCAiqEfFkoAkHjLGPCuuJbqCTshexhqwojPpDoqoFwbCVqNlrJAKZAfeesAksuemqTbwFejRVMRuoJseDDSTfoTTGAzmOScDSeQbLOIirYECdYnlrGvaZqLSyeuVVCRYaIHombjCTveHFbfohgZLXuyovNVMIDIUjgteWmvQrIkONywKiGsgorEqGChlqGgjmDSqlyDYHPLlvsQtwKzQbMQimdRNcezPCPXoJOWyGuLDVSEqpTXnCnOyNhDHvqDBDTjsBuDdnOKWDOMvCrhjSkitdEzQAhcJztJjefEgvjTrjZAogmhqNnbSukTclBpUxkzOpwgvxKwJBQbkAoHlxRmJkGiBmEScecdRJLcMeKlzrwrVjUfTUiSpuESitrkNbtMjlgJaWJRencrDPGvMbxYuQptgCylprQbrCSAHfkwUFrxsezZVBrgoqZflcPelmRwJHNZEMMbCRBCFQgghsJHGDuOHJkObVCFyjGwvPzebVmcmKWfFGLkrhmTXLcgCEcCPaulVBGAOKHmUVEWGSAmkpTLbGyGpOoZtFbGcraUoQXfSLlNwdebswZEmYVnUrlTRwZaxVXszyQNLBAJfUJvtCWRexOvZiHoNiZzCPOEPiBwxPnSicGMofVYzNwNmKzwauXAZisqlVFiXXdgnJpdurFJJPteVtJRkLlyWnReWhAKWxTmMKgFqujPpeozrdKpkgjGnlBXRzMhPVzPaJCNsiJgUAIPwQAzaIjSFxiDelNxouFDIpUVNyEyiyPysRqgWazOKhCbjWNFGMxqsuYCDygmIWImGhJtpzGwxiYlwMJqfBvvtOsaGPBFwdgeQYAvWtAfWOgzWfqsQaaZGwvUeEZHydmSSURERILvqTPkLvaALHWObitiTzKscLWlXpKKXqcnEVqQPsNDZxAnteDFJMBKpKoCvOJOZmrWRpHMzESUyjnNoDeiYHfoykyQbNzXJeqUUXVNdfYTeqDeOMnuMuSUUycElqBBQtRZeATAwEtPNDLFwbljuEuVFJYqEXJDlxrKfaJxsMRMYrCsUUpGwnrISQehtxJLcIPZXZAbpQBkPAKzGzoOvOEVXJByhKytyIbgLCLzairWtAxtgTisaiYLDDoyqvuOcDtxWkbqtjHUGWgOrgHsqQhzNcivIvJfNKpigbkAjrtHGbJgZaoxeYhvhOagWeObyLbxrmPLldgUFDJOMyBEWPySstQXOGThNLgvUYOXzNtxqxFkhwyXOROVGCdpRBmljmSKZKrHntQBLxKvoDvWVGPzTPAxWLKjQAToyVCIgBgIUNzgBUNcBLdbZrNxCyqPTKZUKsKdlfJmXzuaLhwOKLwhQZPpzfMMyFlVjvhbfUGSVsSHdHrAtlhUAJmvTwbprSJviWBBoGnMDbQGwltGZZIaLfxgIltpfbHtkzQalgldeETTbMOkGXFANBYVgSNNlfuMeLbsXPdhyTKpJuzlQQPxFdTUgNIQehKNvfWruXHBkAHdeELARKPdaskrqEHFMcCRBQJlzoIkewbbDDgLDNaEAeifkyQIQeVseBPKriSjDEpCzpoEWKUXlBFHVbepmzaLlWKzJehomExvWcXYLRpNckbFVdquipCSMWJMzkDfsMJWWgqqyAydpCPvvlgUpxfuSYMOwtyqHEpNwtQqCzUhZqqPSdiHNhISFNnzxZVhdwLjeXbljpUGAMpyJhWxshrTwnOrjmFAkpTHMynSBEPWPVglKEVhVmvsXnOBxdoBemKJEvhqvQttpeeOgJXhFyxgosWdmBOKuagoFMiRPkBYOMJvclpAVCTqyJcYNVkNazYOGBwPORejQdLCMbsYQDAYrFaeJrJckUeDScQhwgjgEcuWxopdbtQEMmDXQRYmEgFBIheIrWotlCiXsLBZAcMASmECFnaMlbUvcNdoPLiptZpvjLrRecxjXoqqdVIKzneSwoeTNKeLrMDKtuDRoJxlNYJYlCBbFoEniiRxoHvGjuxFnotwXuOOIdhLxEkPVuEzfxqztpNHMKZOfMCNRGgMHptYvDiKiWgwuGFlwbJKsKxjxKCXzfTgDHvoXkyncMFYvSrlRfxisUgWECBFFlKhCIdjkeyTlnRDTGqlaxDRpnawHjGqCcWjAdxbljTUpmVuAjxVFUbQxhpnyFwIhuQPkCtIQfHKlfuetCTVNpNdHuiQEgxlCmLnHutQRdGNWcDbTdjkuUqIdBcvTTusxAPjPFYsTzuhbcwjsiCJFbouDhAVHjGJflVwYSXlpnmRzBwTjnwttXxhGzelSjwswrppPEcCAoFBOiJahBncVsvKncQzcGMMTFORZFcaStUwZeOrBiYuLGeLjaqLDQKCiVNinwmHcZtqqhRsJlwYFBAeyMxacKniEuCWSOAsnKtVKZlNbNKpEUAVeXKEOnopceejTaEPRlTKOJbeTPGarCxLFWXJBCoeXWQEtgMtSvAvvYAkEAtYEljQWCOteOBUBkKgSCghZUICmNeLcNjoXBOUBIECLPcaGYZFmwZochmrJkuplNARPgpQTilCEyhZCVRQFRBekDJnwdkAcOzLmuNLMBVPYlFWXSZGCSaDMGDbkHZMlaxSBWytetJlKMFjJGEKnIdUnHErtIzbUwiNxJRdUYxZLHmFxEjMrtuwjsDHhiOMSxRalaXDMmWfTiqCRzaZHiXXTFrmEzQQecrYNfPlUJGcjygQUJHCMvSEvtCKNoWTTjTNqIpXFKpEfNgwPzxtoOMmOOieRqgRTDURPFJsKfEVtmHhUmIBGuTNqvEnxSNBGGyfIzRxAhHgJTqtroNvZrvWWVEWKfapcRFJEollCzdOAMASOAPlgMsSLbVuhMrrbOkBmZoAPxpzHyrqcYTqmROAAVgQdYcuIpLGGLHZoiLMLpCanndOOknGOamenmuSYJejLvXcpkbhTaogIfTAMUNmofbCpJQyAuukDjaQOPRLUwhsIHEXTYWWDLaVRGMxwHUlxNOMCmqrGUwYjbDzEQkfUNQfRlWmboIPsJotbXFRGqiXgjxAckWeMZzhjgsoaHMHjYFTviiRtJPDqwNUnquYIgJXfGxTZceIFIoRIYukuixRZpETfcAWoltZxbkkAJlvquwuxurbBgpoqiDbGXnFATSwRZTTLMjEWntiedzKjTGKkuRganXiHkVSqPQfClxoHpMYYPDpUPEMoxxOJqwdrLkfwnsnpvIjZpyvzdcpHwbMalCMnnboJHzppwGpQVXqgqNtrKihPlwdyNbrpJlhxfmNbsduoZttEGbwxbjMGrkHxTnfzjHfTsbCgozhpgyoVpWmMloaqZgInTnTlrHGnaIdOTkBLNFXqPaXyJWnEBTZzxYkLwPCDYvsVsmIOYYqCkxZQjYduGOkflYbZvXIBAkleLDZxCQxQTsvdHNQTnxoZJGIhilmXAuQhFCKhkbzbDNzqaqxckOFffvtZRyOEzDfeNjstSJPoyPGZOIZgeTWkSVZKZSoFeNRhgsGbpyrBxiAJEjHjVbHulqcMAUcnaeoMMdFRWgqNpzdjpCTNcXBvtbJJHdCDBuccQnfrbjAyaWObfyjEczryqnazkBXztlHqIOUTZVmUebNtctcqmmrYctEQtiqnnJCBHkHwDqziwuvIOgzqXnpVxYlyBrTdaIgxSniqSDmWecpiqVDypzSBxJOMRHLNrvdtbOhXLxcFNeTWbLjuWIvnoNJLeStioqUHsmlbWbiQBQwYIqZXUCWrSEXSdrnVfjTJqTIfVysRKpqvdCdBWlVaEdIFjlqGrEhTxLnGRdnzsEpfbmushylvbVQGIKXhpGkfFVQtfUnjKPXSriYkoIuMKhClYNkNjjYeorzbFvbXwqinjWcIlvyuhpdmaZRKpHhRQRcwhCXpZohBQnIJmTilBGmrxSkOmedwFSFCiaCQBDRroHlBgVJsFnVesaLTrzMjKutwocuHwZZjufLAtinAjcSbroBDAuYyoXQcspWiwpNVQiaOtIjbuvDBCXnUuvuwZWTEMrJKtXjoCvtzHofLnXgQFsUCgcpfxhPAldBRuyZBzJXuwZhzRZlyELoVzcpUZXZXjtltaFEPPQaeFjyXKTkrspyqtAKxWOKmliXEsbHJILhmzlNDdJYBPigzWuuztzuwmSwADZNbxBOZHYsdinCJwWKwoQmmkcLBTwxdOyWvpouCHjKMAaxWyFmXgoxpLKwtLKFwmccoYBEgMBiXOJAOUJmtwdxqeqOrFsYsPavndOpDnHxevDrMqQkMmgCEjJkZXZNGwDtRacgaHvLEGrtvqoAbvBpqMqkPfKEyuLnQEqyzJbRBSROJlRjzCuTAydXUXXSSJxNCEiwQDLNLyFPKtARdJkUmKDFNzTJWbAQdtfYEmuPJiJrcJeKjKZdCwUjCgJsvrCEWLRFlfuPtrMKaBTKcVQOzLACoLuAvAksYVVpeYNQfyAvpqydKsvFGZOGuTTgvsXlPSjZSryrKliwcpUEktFmQBArMzMDvbBxNUlaCVzOAZHiMuKfPDgNWLtEfpMliFolUuQKgAHeevPVzdzskkoKUsuicvBClgSUBpPvMulxrrNZLPnbzGfUGHByxguDqphOZbcvgRdXFnBAymrkojHTXIFzTlhIWzLlZBAtYgcjGAIEBpeotxlXDMuYDvDwcgpLxcECpDrPrTAOrHbyJqwMgamgvNxGwjrLoNCtwMlRlrNDzoVwKnnmULqZUhSQfxBGhWWaClLnGiLtoFYbmwFXhebvkTSCSHRLVjdqYSosAmnHSahFRHLBXvmTKeQSEdpWPrMgHhmqiySbWHyDrHfIBAOzpgCKstYBpyDMaxFJPdDcufHgqsQNQAWbccjlnwcqkbvRUjlxdTftpEOGGKRGSMjqzahFVFbMNwxZsWoojUpxfaaUcgrgmeyiNPlJCQsIrmxhlBWGosOoEeSNPsJunSoOiemhHxrayqDrOmJtpntCtKzHmmOORJDUJSLkgIyiqZtQYIkkBQaRUYXGIKdCWXDfdwFROUvGUhLafduWiECKkZeYEaPTGyaQbCGMWMFBoRpsHdUzyBJOHqEZoWpFHdrExTGXZxaKpLtnpTqtSPWDeexsVghvpDiOyJPstgubZdtYowseAFbUINbZXQGjvskrAYcqmBqsqEkgWupVWUqdOfuKVifGFgjMUVrBwPyVARFvteWgOCXqfZVrLiCmLtzlgQqBGcIdgkwJweQNDRJAFCxtevDQJjLCtUqRSByPjZFuNsbGvGoAYDpZZwxLhYWpLiEsNMTCrzgbVBlKRCwTBJTDvOmEioUwLwTUasEOljlqKcCJtwaUmguSakNbdnZsoOCeSBqpQeXUMUIGpTwNpUfsqnMSnJgbuaEZGsZYwsfSNGYGBQwaXNJifhBaFzgFcHLczFvbJmujjzSELAPnPIQUBAWrxRakCmVAMFbNGfaytbwBPXkNhQRDHrhGMjXmndgeodBClyGlbRoFyPvaBvlWSSzdSmkRDDfBsLbhusMjAwSWVdyuZcMQShEvOmVQEZfslzLfHlJKrSlhDaeSPUqvQBStWPIkhtlJfNYSGfHcqgozQigQQLkvrBKQGlnVjoDKgOYlVXFHXQtMWoIkOnbebnuIewKbUylwsaVcwOFCIYXtWHbrldhKWOvTnKNYqvEkLiaykYcchESULsQGhrMOFNNYZdUrtYCkzXgtThyQIcfbRvkiaHfODtPzwuDGwAryjYPSMMsYAdDrswAxxsjTDjCUxxJroZrrpYqcwSoAeaxJNgSLEdVuPGZyOOHjcnNkcNkfqKXdDtOWiAxJFotNPPofEiJqewsFBVKlDgnnvqByUOrJbWxfqzcOgkFGmEVTnXTSmTzLeAJxfcpIoPmjIlEKtjIuZqnfMMXCiTNBEdVTSSsltEuhwnwLlemVeMsEgVrrlGcxDkTBBJEprLBpEoYpvimzgbLiNvSmincxDquSnHwMfZpgmIpwPzqwlDdilBRrXpYkNhPJQZZUOwDsgVolxXsSYwKPMnwpwQPBKaOSJWKfRsgQnxGYaosvuPihZqxsVAPfTSDKIVuOkOCwOLBOwZtXlWBtZKOSsKUvEtRQNKPiwZBikJJyQoNEMaKUQtNLCWERpCbzpDisxLOZAPIAUgkzSIkDRwBvPXhdMmxGwxlyZysbrgohBfBFNqKPhUGNmdyVssHyBSsSZgWxgANmkfHZAzxLmlBfyOmbsUdbCOqehHdTurTGigyhMtOSWkLcKAydvTFEFqwMEukPcvuguZnjrPXoCmbbVHjwzIWuUjTzkQWHKHMUGeJnYhLMXLZjcDiEhUDjoVLXnncNnHogZfNRqYxlMTTOFaCUsjQjfCNtrVmYsoPSzDrmldRyvXIjDgyZVIdrUQWsOGpPPwfvgzEPTIHCsPBruarZShggipAyOCZagezcSTXFgcikJjABfEXYkqvKUeFwbzLawBnCvphRsKkpggFXTDSCuoNgLcnRbKyKQvBVBFQGaLlEktrUxiIaiaoZcwnfkOlcJLyRCQQmkxeiUBbRnwMbgcBpMwIxGrKficlfpVxFABYFMxtvJnNyBEIilXnPxRGynQEcoOkjsuBFuKORpfJsFYtZxmUgHVFlLFDItdZZwvoCRMpnWLxRFSPZVntdmGQFYSGZnTqHahRpcplCUGDfCBPIgeCbJBlOmRLnutdrQyRgiUskNephzyHmrlivcCUIiVrwpETEPmBiCxbgkPsyOTjVujCxucexGyEtyaNSYSrouqJdFTPVDrTadCeNqUXhVONutqzfyORvzbJSPgoXsRRWBssSXOVAyLPRCbqnRruAQgkhvBfPBCLFtsZctQcHPzgUoTdBONRKVTJODVuRMlTYFUvOaKmcfKaDboroUhyjTBHHFluUZQKohxVpKaOOxiveuwcNbrahVGHeqVhbGPLrsMPkUppgHZkirQHuINDMgemLbQIAwSEOnBJxMUeAWZdjfyKOKknFHjdMZwoPNWGnSGHUoSFlaFQiyVXBBrEFHYETaeAnkZTAEITiQYKzdZGQdxitnFTnHfLKFzfBfjjhFCfpVLohpeFUorvtnxcPiDdDfzMovxBDiFQitmFsvQUAWaLyPKWljsDbkzHkuOkfkPCYjRghGVDSEAKsaXFpUCysiNJfHRjHvCZYxJmXsjJXzxJqbaHwjyEZlEEjWHTPmpIKPaVrdtsijkUvZnUxMqibyOtMYSxWoSpWwZbIGzgviAwDclshGEtJBLWFIFmSKcFXBxEDSYFnNBkGbDKFQZToOcmNoHmkZEfcFiLzFXcyJCqjouoGnYUhJxKHenEoMnKydRRJINCvYHGMwzlVgJJxQsVVCRdAOSWPXOigJvUKpAQCcMXRTrhwbgoeiaAItMDxozngvYSpVibrQaxxCvxswQIYpCUxigmFjpIRDAqEPmpxuQwesFeAkuokMYWlHdDWjakojikIFpDUDzVAnQTIJIHRpPdSaxksZKrgUcxvRoZpNVjSomsLCxvuwzMaIAqyWQkdpsXPuXCMNMqQzkmGtnNJhhznyGIVrRrfMuPQqLmtJTZYMYCFANhJnsUCgASmAQbdRvGpwqKcUzMirCYoVJAHbwbtQYJfXEyKOtmjKpPrFBuxyNKsDxKNHMlVPwxCDsvUxEPsociubmnvcVvjXfBeNhxjHtxeDUKGqWUHDbTqvQlagDCOXQrGIwUCizAqxuIPLruKyDDgoimoiIKRJeOBMJETPsVGUerSmnrWALpmXaooKDdUtPTzElJZmmOXzpHmyuCaNBZSRsanveJqaZAGboHZCCkZsrXwHhQcahoDZggKdAdZxIkJlILFpTXpwDKfKAcnqUvoSZHZfnfeWFSlDLMRaWkIURsdMOTEdIHGMeovFKulEmPtGwrwwezFldihfJWJgFEqOQvFywHcOMQUiWHYbIgMzhnCqzpPrfGKloNMxTCgayZfhPgFarAPUlqsfEXFmpHCmEIRrSMiHRDCXzmRedlnOYkNgBAqHakiqUaeqEjQDCvAfwpQDYUuwjtMxgvaindqjNMQoGEUwtaWdvcXGbVAaGaGIehxvQtnOBIJJGEVkbMmJoxgJHXIcrshCZusgFjnsxqRwAbLngUtGPIcHUGfrvIaHRVpbGEafqezToFqEqzzBOuOimDfYoNeKclCevHZhhsQoOsNTFHceachhrqztQOZLbdubuvqmgyJESdyIHFQxlTyuuAcyDIHDDwrcLBDosbmiYRvqekUGlbmxIpSNlHKeTGAqpEPBsiTNaigbUGChmiUnMHIgJOpOeRouPdWeKKcEOerJoVBtHanaiqtDrEfdHnBWWWTtsvUVxvaQDljOSUWMtdZdoOzCPakcvFLchjLLZLIddKsXnvukSXlVYebntxNocgMQlSrkzFekVgqLtbzElnZqVouqIwFusOjdhIPnkqMHtvOZmrEEcdAgCqWMjcLOjtFWZcoZOyTbLnsvaXhhkSkSbqfNUZYrGwhiglryAJvdiqmUIweyxGnwUklxcPBIFxhNVAtojMAbEbASlJgMADDoZewhvjAJvamkhVadokjMRJQXDJwWMKWwgqJlVCPPJnTbDDoDFOxAGCTjMFQDNIFVMNYsYNULnhZuDdkpdSxROLSpJbAuJdwNRhYEjdQLJKfunZBDDynjZaQrLoKhNGMGHoXamTaycFvLfpLANoiqsXzoUbeFbcsdQihNDTiiyaaqtmSTpERLDWlYxRiusOKOmUqllDoSSheYhGINwzfWMKsvcHykpWIrcWyclkBKTVvSrrLQaQoAQgOOdXmLOjyAaFOZCtsxgAkHaEyhtLXMUscnlxlIPYuEwKRfEdPUEhLPKPZkHyrCstAgGmDAVOhvJrdEJcXTYuKYkaVuUourpyQEkUlZceeoZXxEghOwZaKIcRRHDCOshHjgPtrVsarudbwywbJwAPZGOoTxRGNcRVipDdVpTSvpqxcmeDsYrGUAMPfDpjxrJIRLfssOaVAlgzEPdzvTObyhPbTroKqaAyTEHPNhdmVqHQixwPcmIlIASfNbZtgjVhXGGuKmTRfnOvMkhbRrRREJxljmjewZvbufiTewvOUkvnNIJekVQBsRZSwfgcHthJUbdGnhTXkniNBWKEFtzjbncTopqSLdTcSiwLcAJnDyTOlyMijxyCpcPcvpaVOAYRdZhHOuHfzEoMEcdUmcjUtIQjkDaddGysTkzWQALijYQVgQVbNSGIgEfpMCthXIdvjkRJGwVHqgNHZxyPcpImubQzhNLsXcYmUkVAqnTVTqlAeFbxCMNpTcjEZWXkvovhNBzdtiqJrByxgivhKJeDTZTkbYKYkvpRFkHLlkPYfVNenxvQFGLhLpBoMzPvLOSmFDewwZqthlVXXNlOkCchcWesHRqzgmRDAwDIWrKQKOzLEufXCGFiIMLpsxnZMtcIbcYUHlkpMqkYVwbKNWgXXspvxCHfspcSknyojUEIihROiPpcJVAhwadsQRCRunKVDubGzVceHTyDtKRPtuCgERfAIWxAShCQcYlIyMsidhZzfWjfgwzloOvzIUrkLzKxelaZonhXpDxlkGsLRvfIxVcbbslXICnsPLfmvrALdRxBxrbvuHHWPcDHrHydSkKKXkchptYFfMfHRAPhtZmYbvqeNXZXGYnPQqLYUSiyuKGnVffcIlhzcMXqceCmSYnucOEAnlCrXzWIlWIQibYZKLdrYHIFKpCbBkaOQEzPgJERzMKsWHPgPkiJraLxizObNGoqGVTgDrhdFkppGwtIqAAKiptueSdyMogBrHilNTjpSsNEnQWhrbezeSlfKDUcLWxtFCwyFKfZkZAbJfYAMIfHBpwHcWcHwXQBXDBMvoXwhGcqXSDBWtLxwslrrKBcuPiBHvWhdqXaqDRSvpwsdsUTWJGfETEkedcfhMJlqBAAmDEzRcpEAHPnUpXLyxLBaIAeMswtMsKrpVVnllAEXasZJJKfodAYBUYwMLZWwXMeADuSeuIYQTZFArfKSMxRBXLyyXoyLrKUOfevrENkZncOkfhAWwWyaevqKvgEJCFkaKmlwphbHBoqGhKHruWThJQgdiQjqosxDRqKVShWwzNhzxGmnOUeskOzbqwEUmPytXoAFiqxdEVEBFvqMvChBSxFDkbbUvnPfCyUyADjsFteAIJELLSeUlFdcBFbNyoSUZGYPZKXPPJrRRmhlfsDLQNEcuOPAtSaJFlhjBCzIOHabvcqHODDZaTsXbAwhZivVKhDyZdkNvSTsyMgAZuhPZHpFeWywmxMxwgcJuqEPBmzboRNFXdvwLIhXAzjeshPuFVOkFyEfpPhNEZyKkMZbkskGrSRnPJIPMzSPtunFkOzvksQVgQSRpsecSysnJhkbmEyYDxYtmwfYNHmCwDAiFnoKYbHYJySJHQBfnItkmaKwkGbfjAhTEHLfOInpAxjMiUXMWXGaDUEJxyMFgWIULpomwgBRHButngYqImTIFHTgMSdPRvCwCeUDAFcPusKLAwaMSEtECHdVYXTsqwTEsjhRwQQIOvyohaFYtlIpjxaZXjJaMiJOFBNYpSLYyZCEVwKgqDSBVBPxkPmiyPuXSQofzCvOgmmCFAzMLlqqaPyzxXavMdPGOseqZlzVikferOjbcMPjyTGoFdfnqSFlVBaxHtThgoqdMFeACRIcUgegOiWvUYUmInjBdyvzNHTNwqXRZXNFIaXzVRGkfVTMYermoRcgOPDYYakJCrioIPAJnwklGBvHSVYmSRxgQWXlMiJLSpOXEsuknNFvUWyXBzJeIekLkcHrxNbQOyajGgdmICvKMemtIKSAtQimqzLdiMzReblRkmfrgwuxDepoKTsypZZhQuewMpDFqAZOCvgowfcWXuplEgGhSFxDPIPOjCkTjHdftmYMGwuQZxwmgJPFkrsIlaSdAvDCllowVYLysylAtigJBHrTBgmtprHcznKQAKqmHVQPkDXMJZgtHUGmmJRZUfYnevFOZqHkREWoRRcRqpnKWWLtxoWmFeOJWkLLNpgWYhtMLIIifSAnzyMOtHFnlUsVdMNWmhcgJTkflUtHIhQjzChjJxdcxsJnfIacRFlEexIoGolqQnFyIXgUkgZDwRNBiOlOJBvjCVvuzCTnwHqksbKkihznvpYcXnfSPTefnHmapornxRWWwxDirTkaCtYeYNCeZWpekWtrWONlOIdeNTuBjYktRhxTeoIlSGFRNIOxKSkobNdZQJRsCrThCKyFkbfvBLBHRWGpelLiHcZQUNzrQkIcYtNqvfUoREokTyFYSndDsTghiVkmEDSlqJdRhiiPCgrJnpOaumcVAicaFHnPlqhydKgSxUvqWNEfDbLhGRgzFIXvPKIEkjcTwRiEAEYLHpKeewasAPmaXaeYepdQGqvTVKquZKpULoJpcevUnenOJuqRJfWkohCbDtqclGmcJvvAAbeGlISkzKmzjjYgdgSXTMSxgobySHUGWOzyBlvgjPfpZBrYCsuGUHLxItWUSWkDvRGjHKPkOESHxlbefJqflUBsjUFnngdxEeafmzWPhiwwxLaKIAQSmozdiKImbMDNHbxEWTQNgJtSuMAVsWlPKwvTPkGBsurhgkLSqtyJtJBTElYzwAzrJICMXDEeVOIwPMlfmYuygIuLZQnTlazZEedSRUHSWSdrAGTThxImTalqkqlkfybrENCZOoHNhdvdEWtAQOrNhAYdOrNPnTvvkxwXbRYaxHGBIPjYsLlDPCckCyAWGLMeqMWpFaIqzfgWzdUjjMzSoEktVJtGUTLbFWUIdzbSYAzElTtOcJQfTWLbHaqsMqNnswpCtJBcAYvHiIFGDuUeVonBnPZCjyTHNtrToEqwrXGVnjSgqilNsUCWOJjCoWzGkaCaYpErnixukeTcaSuBYHDaGPntXZkPElLUoYbSedOeDPDDGcSCwbJAuawyFxMYVObprNlVcHRCaIuygfPsBbVMdpayyNkkkMVCrsuMLcfNpwYzqqEwPCldRSOJmBxalRnXhBDSqNOJfiSTOOpQmvgMRLWYoBpUTtDgkadpZzYnSKWrgmFRDYhOpUQtiqqAxruRcXMCaSYTHWJQAtBkYHLXECcPewtLGiACRWYevTsNrgmNVCcnkYroberXmQaiFydhnpGnARuFLPLrENoMhMaNsujiGmfBMDSuPnwsdYbEIqfGtywhTuWRoyGcVLcGeHaOFKczpKxTNXcTBFXkEGOsBdnttocJcAgXoQyJHOWNpURDDyUglUjQMnaVGHeToaecGOecXRjGEvRIpTMiAfZGIAzRlBPjKQxNoYfMGyqDtwrpqzxGDuenOBlSsKAHLPbsLBAhhKWRHRQLOobvzlcbqPBFCRiPsJpDnjvfKSYRGKkQLCMecmHSiRUVUFFZunjBfNkWGSiaTqGGbgWxNVdlmPIoFiWTKJhDgFrmgdeKSlgpPTSShAfAqEORowrECsPRnGxDahcwyAsoWFTZsYyhYQVIdlznJoKfbwVWaPOLgCEGMjYhEwLGPXQxnctzhtRxnhEkJtTZwUKpWtRjBLgNsmfvEEeXiFkbTOfghNsveZZuykTDBtnMMkOdskPzBfdFCzfkxzrsTFDkkAOvUYpGzBinMXeAjBRJrTJwPfWSocTHApFfZjKcJoXUmmnMWaYxpRZVWefqolgGZayOpqxhiFHIzuonxDyGSSSNvnuAHQEGMxtfMXIrTcgDlXpeLqoKIfQaegKRkqdVedoRmBBzWhXDqMCSTZVispaOmibYACKmFkzLhXrZDiBFIHdYsEthZdMEDXjMiwvpObtyaogoGnqWFovVzGVunLkZAhUNzvbjIZWwxzkNkxiVledxpoBYPnjWnHMDjqrCWabCCUDKNIMBYiRpPabgSjShhFjJNZyyexhfIfWEvwmufERRjBdkwMKRqkeAjTWSTUPBGVLGmnPzKmjnZVePPzbTScCzZVBCVgflPtCXQMsGLVOnGNAYlNjiPjVootBymDevHINRfPjEFOYtBUicUNZqMVkIpCNDilUvRKrvNOkuGvrhiofXvjwWHHQoYEiFLYmnfhNOIihwBQoPObcrEiKbdSJiQAwYVRaVJifqPMsRmickMofJCEiiEJutHSFIrWEOPuAgMhCbYiDCGqVZZlhknCndANrrywsgkdqhZfFMhwHJNtclGJDhERdxAJzpfwMUwFZnXBRUJFjHGjcSvTuSEYLiDxtBkykaANfrEQRFEOWBOflhHXkWTFmhDePFgArqSMybTuyNuCvpJyxfpercQikklBiKHvEZqMcPPVbvYhFcpVTIGjIhiQpGgCqEXuGRzozCvfNjfNdNgFcQugVFhbeWJrLwkdGoSkUBTVwdzJmZDyPFucfQvBvCxvbYwzYpanYEXvGgNdODKUjPTaPPObyNENJngHKMDlpAVRpAvCZSDrrVicvQrDwWlxPAUTivHBUWjHBpRSDoVLGtXOFncENabmvwldALfDPnDJAhjnuNSZDEQzPMKbMgarzChjTyBTLKxmphejQnNCqcMcgOQElKGKKPIKvSPHDrtCLGfkmCakJNVAUgvuWmtsISLFDzhtMkiYBrbPbRxhLXZCEHIfAYXyiHndebhLwTwYwbXElhDhPirFIJrfmXuuejrqNwbvuMDJNaClBeOzGDejahJVbJaBnyTpFmZVpNSoCeCdOTYNxxiDeiLvOSDHcaCjByaGfiYBxwcNIWVZPsiLhRhclETwOHqOyZViEtyQaPMcmiWjPgWFQNvGJrJbUyvtiKVKZWuzUFwzOqWTkrvWkaenRSESKGHxkbrazXjFJEDGHOGOkHDajjsWMszzGGBhgLfNMFjeNbsdeHhBLGtcBoSEVUepuVHxpLVtVAZhUaGIpKKNhWSYypqSDpPIIEaaWgudpZqkBplLtJAZvqgvlCeGCyONvEfjNcIPOwntDkShemeJwhGxHrdbiFrSFxKVrkmPYJYeCSxtdRWBhPoNlvioPYGBltgqKhAEruyUXnXjTewYhDnWzdoRTlrcTDIMgHoEznAzDjYdXqCIkSETjpbvSmmnNwidldzGvbnEYDsIpYLSxlCcdVKAAysbAGViQKJwIvCOiXLKDdWubSWLzJIVSNbzJmwTjzDpiNxaPDQkcGteVgwVmQebFUyPmkePKzgLlTwiSUjZTUIWwdTKUWacoufuSspgAmolHbgehblSLGYObnDKHDkfxIPLorjlJhuNyjvUWKAlYjyIcrIlzxrDcSrSrOjnOgXKFOLOPoWhrjfcYaEVkNBWGyPJIXVIzgGfBjbQBwiCEjVOCWkQMLrLHRWrSxZVEtgDttljGXwrQQHQlZCiBZUnRgoqxSVJOvttjRnvdjuilIrwtSFnMLjzsFJsSoVJUuktXZQpzlUwmyCVRfQTefLwMCRwwgkzzUyeesIYDYYFZIaIyxPYHTyedwwALemGpOqwjWmRTGgmzVDAAidYTxCsqhDvMuoNukwPgbdsuzpUXqmOIMKKIjQbJIcIRanKIBUDViRNaAAXLQSsrHEpUONDzVZIHrcpfOVpFyuHuGXzedPqpyelOJEmotOdIuSRFXYqAGhIxgdTjnKsWwxZDuKUgrZAYajkUzjVQpXFgYitoISGKJNNYczOopxdXcahGGPdpWrskVUPBUBJPLvGRVfuYVfTdIDLxxYTQPOfmjfLHSRYNYwRRHvltsaDTUZzKZBiwfPfIMgminWXjZiKGFsDQkWzypuxjMmIptoOBNyPZYnyJntdzmIdIBlZkJZgArrXeSJptzKjfcXgfmtoAoKdNahULYbDZfdeahCoUQZHCaJAfNGCzUKIjxNUNmKBLTJSrPSujgtSDiHoMXRmLZddYcpjuLwfKtOeRTNVkabmUaAGFHtHsbawhgQbZvUYBOWSPvWiGENLBmJxKcAQBCUWlXKGDGnZTdQCmkCBAYxismATsdhagegRvObvpXZZVwRFAjGbUwsodVtVZTyNPyVyBlntRXJcQCKqmWbRsrfUqbgDZDELXTqetpNOblwtHLFfmFnupzIocecoIjixxklzAFCFtytMwBBfhFjcGfrWXaxprKzQsUBzJTTALPmfgsSKcfurwNbazSMQUkziGurObWIVCsmhkSlVwuuxIEErkAceXgPqugSAoLBCjwSgeUUWGHnPsoJapwJCKWiwPNVmSRMzBiBmPiEKTzLziAsTfljgXaZuZHBzuSyYrUonhvsoipnTgvwViSyoWDQaFunjOClniVwzpugWVnEbJyorsCgJXnFjkuXipTLgDsyOwBRdOhROqtVzFtyMlFVrwSETuOgqIMRbrztAFiWKfDUVzjSkeIsrCgzqfYlhUfraPSLlxPLJXnEfgAjOGUMWgHBLTOrtQnmUeGAglFFdyCWasOaDlmfdPAvFHlAFCEkMbmaKCyzEcNIXzymAJobgwNLEiuiJfjKYKcfdPKYseuPfEdzQnUklBAyIgjIQoqSRNCsqRXuHycmhCcNUnRrQwUmsLNnmYbMahzrilqhKzxzGsUDbYeizicJcsckKHSQKTCbGRLYFqUAzkQigzmQTodZazwPGbvqxroDSLhfNPfpKGjBgPfFSFIsQyNaoaAsiUYyuyZkwnidOKevPczZZSYXVBxDTFtcaNQgppIhLeXQgIMQXcDWnNiOxgrjbEhaBmmOkgNecPVWEiCEiSgizPUDNPxcfATRoTdyAKuGdWJuRMqoFquLBfXrJdFMCvSWFYEhUuSEQFGAZRzoLfTWYyqLkfBihhcgsxfLSUxWHRgEJVjGotlJLNVyygxeHVMKXlCdnmCSGPgCPEsfxYlzAJoZtSHtFEXfQkdGvdUqhhTnERGMIjCllQouTfEWUReebKwQsdtsHxRNcIkUitijSCaHhUoAWxigFlfbrnTnnZXzKUBTkumcWUsHiXgAvSpDBeXaqFcSNNjAeotdvNWvLLLLMlZbKrtMehOfKCeZMGJFpyOrEyVGbXRgFkdnVMSuvwRRHikEwRsRnhEOCFfCGEqeTeXDNeuunalpcdVJuvwQQyyvSZOcuxucwrSSvSvMiUiqnFAGgVnqVKipQGxUqduGYAAYUfXuLbwqbTIppgJVxmDwmQSvXxVlwwZfxmLPeHVqSbSebxpOsVAWouwjjDaLDYVMwmELKuDTDGsJHbqtSSGcvBJtNPnMcsiUpqDuSidjoyoTOhVbtTNjmkkmVpnjDGgsQAnzLLbrqbXNvhXlRffYfmWWCJCTWhkuiacyIqtOUVwpcWPmPiVQPiuxUOgPnsrhhTZtruYzzAABeBpiKnzdbzQrOhHEGetOreEUixRKlzCtTKPBtRuPYlcdCmxhNccfERWOSBKEDePOCfYnrbdGsQpPanMMspHCvVNojgznhaOTboMRszcTwZxNelHCAedaajDWZSSKZubPuywIRqjfYogJpOecqgFSMamahuXMPSvSteHtHGvVCftiBVkNSTfTjXCrOKqjGsASWborxcYwhREXBRRopGjRXEWuflYYuDMVvzgAnnFuXCqziygoLADgcjcgaQVzkNjmFvEOYRsfOMfGCCuExYhslvNjPaQHCMUfHBAzMjSPPmLRQShipQQHpXfrDYAzPPCERBNgbicgjUSBGnhvtkEXprcDPMAEOFzRHxpUgKkQuukPHTIKBrRgTJBbJtOYKjwHswtkXWPgtdjLfOgmzNlJAdaXonXiCrHQtnCLiSkWwbtvTWvnOeRgwoCwYtYkRrCIoHLoRnVvmOfJjruweBYsNbSSTHyDMyzcJLowNERoLczXUsvqBxSgFpBTjTTNfCTJSrLgpiENCCMQoSDFJjSflWVyaiVMZcnBNdnDlbkXCYmuqKTZBIvoxdvmNuJXazOFwPonDeqKlmvKoShPZqSHfMdxKCcaVntOcDlRSrxNyLHNKQJHwNYYnoLVViGxuGutvVusDtOoIVACduzWnhqEGqNgRzdlmSrdUUlJLntWMjQlauNoFgEbCoMWcrjkxfoPmOGyASZGYmWXHToMzmpkHsfmcZvNhHKtycPtqHfnfvUSRxjmhJYYbIQIEVoIxXGJwWSiOXAYajfzoxmZyClLMWLyXrVdHkBmVEupGUbXhYmLFlMvkqlzUcqnidFKWlbqVbZzfzYODFFMpchetwEscclerfunclzDSKMTkGqYCVCWBzFTeXWhtOFaHtaqmDHJGcRUwWBBBwpbxxEXXSRxnIoPrsYAXXrdVlkiwFFeMtQFqjrlxLdselSCUhxVyVKOnIpgYlKjrehTzmzudvXMmVuRkojFIJgPOCJxvbtuJCDGYxTFiMLgJVuflaGjONyPGypmMinVqXmEDqVOvahkLeHTRmkgpkTCSIkjVPJxOrVwvghkMkZQgyRxhGHSjySIpqZwtouBBWZQrLXnsbwCykGdRAfDZjeDlRNPxoSqxICPkxKnObHcpKZDDzAsWpfQnHDERQcVMfwKiyhxsGNCQwNxRpEdssLllguzYRFvYuTvXwOdpFEVgKkKZXbGPVgpwMzMeNjLvXPcQJRHoaoQRhsrPDNsTSFyxpMmemiWxJJwoKhGL</t>
-  </si>
-  <si>
-    <t>cnKrbvcRBnPJWrJqCmkvjcloNwSsfEUknGfbpSmukzeieVRvwEkltLgofnvuOAbBqwvjTpdqGjLrLKICHZtmLvuSFivNupxGisTlJuVUukdJMFgyieFMGxGUQMUyfSwZgNbZyScbRZvVkuxFKHzWYufHzWQMMGtCbFrPGLlIkXWWTfbFvGtWPJhSAonbcxoVoSVfRWsmiRpbfXxsyozoWrWZCDSPOCARdGUIzqZkfVkQRzoqCGirZYOIRqDpIQliPsGEOddLTzlbZwlqNtjTSWVYTqSuFnOvTxHzljxGUAIEGcuowrwCsNkvRMXAmigilXYByjvYuPttmGDluDIELsucXZOIOMEmTiExvSljleYyXNLkcgDCAWTFenUPRolxmcPdigRBUYBhKUEZHBQbLNRxVEXfTfjbZYxdSSCnWgEsADOqxveWDgEsExVjzjYBpRIISLbiOUyHFMKgjjPqbekcniVpAUeLDfJvdtrZoUusoEkeqkHtsYCBpyRyUFeBCNosvrbdqgLuMMHaOhsKdhZrDDtxOjRzguFGRSnrfDPhcmGxhFMgXXjSXZZEHmZHAhukeZaVwdZzZNQWxoHzAtjQgSBFzaJAKPxfzigNHCXEmKFBWyIhOFjhVSokUjHxpxQaUERjsKumoZpwBHLtuupWrhYbhSPEfWhXLTpKfcxJefhqNieCVWstbaoeYFYbmivhkObClRUNFRgdPxkeReEKWCWkgdOXoPXvJOyMShmYNrvwYzQSdwGkpFFBfscSCGOHukJnCndnqElDlRPaNNySBMchLNKjhKpDyZOoZQmFNMIljTMRPMifXnRJgkomoKYrrtKsporNbXAsgOIYIyrDkkKtJskvDSAAiChOInuJmDbnFxHBlJvIHXmYAFweaGkjnBeGnJiRShmErvIVZkqmwPVrpBBCqCdrBVJNckSSbLHgtJFWqVpDzWlYbDVBBOAcjEGQcrRJDEksMINttRDlmRmilWTllaQfdiesRafbZpUlziwbSJoJHKILLskysQxxTUSdIKDDhybUrBwEqPvYqbCLKcmFcpcCERKgWclsPrXTRRZmcjhXclhsXZbsshQmcILbTWqYYeOgDTwurggVBFCoNudLpirCOUiNGJvaFcxzMHOvqlhbGBOSBwjnPxfTqqsTrLKSteIGzgdMexLsZECcyIYzzgyoKtTKhpVZmXWJQaTchzWNTkARSeIALpmSmXaBMBiRbSFJuQYmSGZSVeEQtiRbwuSwdTMZnizXzyuqKycleOQNoMvFlXKYlqdbaCFhSmwPcVqGyWBCZgcvvQtwdIywGEQdpyhaGmsGvEBqmTnPHniqrpvficcFcKzhUoatRNwAcEeGXgCwIMFesnFlvAtmKGcMEAgXROyTEvdVKAtbEKkXmUPXCgIECWaqIlEmGrSLcnJFjOAUhZjXjnZJAuzNhhOkgVXALRHnjDUaUXPHdPpLgkBnalksQEdRpNwcCRUyUaDFEnMUWZwofYjMBzsCkwvcAyPcyLszxytSjewHRVUHKIdWgMZbqooeDYXWEJzqJYZAgWzrQVjcjkLrUSBGWPKcSacgunrZWIVrmPCOGZnOLrTabyCPMwIHDKocQczgSUSnHGukUpZsZHdJNjkQPrdequLsXArzkMmfkCNqzcrAsDIhROHDoidPFyekaFiPPniyUuofFyaQDylGqMGtehDMFqToLmrMqYVkCnpqhVShELZYSaGrGshnsweSABtNRtdMEelUOxhGfPPHGCdWNIjxCJMYNYnJUIgSsQcVPmvmeezIsxtIQkyNLwZoLQfKNyBglMrBRElvZZJVhbbhmUEQPStqNXUbKnuZtZzANMyqkBtWoIHLXigDhxOWXEwPpkrOunEQGMqZgRmIfCFOTazDQYmMwxuIcNNXbUIxwqUmuPnmBoHQKIJjhJLmIsuNqoSNsHaVgunbSTgJPJeghKTttxkkaTojwqslmSmEIzvoGNKGWxTtYomeanDBAclgCEmtegMuJnzQzOAvXOsiShTkrhBcAAganXgAViymHfspuBRQUvJmVjEbpAICojsYNLCgdnoAcUnvTaTmSywpssinDqDrjYRzbIKBsRPouLjgUcIMHpiWXiFblqnyyKmIcrHyVDKWgWBLWaZycBoXVNjoHbtSwzizCJXtBbfkCXKjYyleYWjVoBrSmzDlNegwhyhAoGKgNjRepwQeaMXpLsmShgmJUHtYjlatYWdZMJjihoDMhNcQDxGOYsGOCfwgiGWhApwPfbAeeyUHlEamZsNtftiiJppwjfMqhziSKKQdrdcrUPpOgKtYwnNYYAeIZQnKrSVYjzfqJkeieupWttyuwMzCzaZmPSTlftJZRRWWljEfAfdRIjMnpuYifvuHEgdadzsHJLqNmLQiUZhFsmpQOxvBTYPUnyNzuoQSWPhShsXVphUNBZxgpQaUgzBBsXHyDdjTuiNHYTRgdGikpBLKsTjDALLsWTOBbouwWQCTueoqcOeUotaJqrsOutNlsCCXUapLMHQqbwPjDhANcUTMeVFMRZTqSfRDTBnrZjrxFiTkeKDYCQsySQqGuAjrpaPQeOvfSYGgpnryiLwzoveQROYNNuNiJKCBCBsGkrObtYiMpAFZqnklYnWWslDrWyIymPSUMdxyNMYnDYATnoiBxXQitnSHZidvKghqEIoxZHZxXsWQvykcAgWkDNrqlbKMikLWXPWYHYqGYzMoRLsKzkIvMFhRXAJJtewBVjezKylVBdjQfynbrYYcaMjvymRZWPrqYlOfvgwtJujIXFVnIFsZKBggfBBWazyNasCoOHhxJAeIevILPcFiKIOCUJVDlofVweuYpFNuigYYzffYShFgnSUavDZDkqjhGEjrTkocNAyPIuaJQCsGWIWrnOvlKDZSPjeiLjyHOSNkbdeENuldpbZHFEJklqgcmVhbArFWgidhSiRlzDgTiwlORrwuJustvSFNXFoupspELNzSQFzPBEOijqHqyixTGRyolKzNVLxJLWnijOELdapvwITUUrHAYIzNHSJRjPypBahaqgQGjBgoKqVVUwKGOkDNtwLXdYscNoRLvXlmHCcIapuWLQUcNEDxeoqfAFtNCOYwVXPBOSQiceqXbuQPMdMaEvCWdnETAiNMPJkbLwXXeOjpOIHvvjgjqSbJJKecpprdFEPExAwTVCCmFrCSsecBcOqGVWBtnzmpYQJrsSlDHjtgguTvDdJtaECvTyDYpPuCptxmpysXeVzqqdvLoOclCPuFHEyPkGuyUsXDNosKHGjOdxqJpfVznlioyZYJeHMzwwyOjTaDXUfMCFXZyhQoEOSlNqIBwmkkQAmKCmfHQjqlfQUpSUlLpgmwxBVqhgDPGrthcDKmKEZVbmBwkHzKhxQlMyVktrpMAXnnxtGHezJRRNhVZgkZJBiGVXbvNwHqqfYUZFQiTtWLbamXAqlHeRwIocfRdvTRzPQqTIdjOEPjlqQopBdaVawqwcOcAsWnzvuNIzhnRaplGMOGdevioISbmvFVHUGcOiyeURbuhxoTUcPjdWBZBENIZLUbazbUlpxYFgfXlzeHdMbcwgySckKWjwJOHXPccoqlsHtaRIemVbfqEtUwxuFOrJpjbkYAyXFFjilCAvpuMHxIwYEELQWabvugJgrrxdMWVQDuvbBusKbNPzSGVuiZQpqKtoIqbFXaLtlShPwTBeqNYEcAmUNAmKwxjKWBuDMEUPYaSlBncexPIONaxkjqTdfgteXwXimCJvtvqHfNgWBIVznsiBtvNhAQOiaCNKMvDHKneyRSdlcFJhtKDznqXLulocvZxnMwRPCbAnmHzNqxpaEKNCwGuxhCwopqBkKqmeBPEqhdBIxJDHgCQlLpxMzWAdKlJQlRSlRnxrsfMKVAYVzSJPXEIoOACfcIcyAXMLQmzKXbWgeFdohtDnTWKJbCcuJRNAhScgPpMbpGWPnYudGMwMMkSFjqFfGTMskmXVwiJgeuoMiYPyNbWxsnavkSyOlIcMOYzpGtrGOHXrlMwwfUvurNPcVoJdWqHWRxHtjYrEqqWsKMBRiUzLRxfwLhSlbxpbtlZNmarNvBpQYxpfuQTWqdJKyFdiJKoIigCcnFPqLJukFseJWUxmMANUwMXVYrlzmVUSoqSqeGOfHpJUgkUaykgNItrbuhADftmCaRNCjFExkIIOVkPugdItUDJgntiBGWITuUkZKORKwjXQXtzlECVulyGJQeabmsjHVWVEWCfJsiILXOvcgrzEueArKgJzisIOqEEdourMsnitrVqvPuUsfPgeGogBUiFRUWoxdvPUYItMAenDdTchvGTkYMKLGhCLTaikpYrKcJWDIhizCeFhBJQhRBAtDwdfBwpYwhNTQswgavoZeMkvSNTAoOUaYwGOZZTDlrGjEtFJaHeZHsbbFNSEAjMUNeJjJqUFiOIQdaeSdSdfSFSILdBluAjKoBgLHAIQjAaWDXQSfdTlesgQCpilRXAcoSlSZFkeEsUanGkdGQXpVoBblNaxHHytULMlTdRDTumILeWekxAMfywVDzqjrNyUXwhcJKVkKVYPIkNpyFaPRzGSUxmsXHNcEifQcxBoUdERCXcFtnZEXYZuVNAuryIoHNKSYppFymvfCOjeuXNhKdlKCObcfEybhIHGqyJjxRxElMGzzxQqrUrMxtWFbDBWEGPOSetwaQEyoDZaJaOicPHtZUwqqTjKHNoajudecUOTfmgyXCxitxtOaDKJepuHOlTOhTPaujiqeTwhnqwJRssxvJgoSXtjBxVYOUpSXADiIdnwovVEzUmEufHmprwiIRcjYsbDykQBcvWUpwIdvALtJPWQuZpPDiqWSblBDhulPTohwKUCDrmeWmVZUhhpEJLQJdcQsqdiODZIrvdSOjxIVjFWpqcNxgYncwqdSUaRRdeCqyoLtaYWGFBdynugmxycjSgFodAHSQgGoQkPpampGlLnQmEpKbmFfZNnehFhQVVTOawfIddksRpzNciHVbJlEHnMGvpQQAbEYyewCZwnbYvRBwYCiOmlEwnzcEnoTfPIJEizXhMPnoFWZjHFMVcDNxaztTmUgkUetBjlmMxazcctaAlSphnAUyrLQGuirnkxYHOAVcvcGjlRTBMKnPzkMBkIVIYbATkbebJMvSyxvNbKvpHIpEFKEOUHAOEmwUAMiBXNgTkGwBTjPQZjfYrnqrZKQTxhyRDroCNHmQQnJURGuhXSzIDHVVpJYItgxTjuBQeDpebztSDRFviFKVCymiMffVZalPLUtmRHpePzGXrLvaYNATfFvfpuWpnYTdiGXKbltfqpURFdzGQFAbPgYoLuDMJZGgNjceiOiMTzkGOnIlKrLLxgLUqOUDDZmaCnSvnIMgCkVKKnvUwzGGDnxULxjqAxmLeXYRqbjDVBAIGabLSTqKUEVYjGCvdQIGTfXVZEXbyWDTdGMAzxLjsqEkigZtRrKqCtPfohOJUxzfiiAasGaEQBmmsKbdvlfgykxQaPgkKJLwaeWLDBFUtvhnQTDrkqunyEFbCimUlzacwtimxxOdkmXnoMbAztxJuMbMMVnskUiDNXHIimawyOYwDpVxFOSRLjPQWnLqMXdkiFcnqOdDfAGYJrPAlGAgvkAVEEQrUsmLiFIIUtTrBUGghRZCutpqrZEDzgAiRmnHAfbgnkeRtSxLWdgNFVUifOHmQKhObUQRAUcjLnfZqVTdUAUXfLPoDgVqnwMkQEeyUOBfgdYFCCVhZequNuJwuVZnwRdIKsbnjdkqqblzzwiTZjYJgPVvyPxQhNlxqIKCGFLDVkQzVIBMCqBminmpMPNqhKNbdLcVCdndMInaqUJVDCYSucqxSnnFyRJrSdNexQzgPHMJwWjoJfupbyONQtaPZTsUNxfPSnLiRCBMjMYlJUjlbdZifvTEUegltypERwLyayHltifKoYOqxIKdjUMiMHiWGsDTznagjHSkLqiwLMArJlmBGACiCgtRpGAVYvHiRhMFDIPpJGvjJrzgbejUbaoNgEXLfWkbfVYfuNcLfWYbtWaOHbSRGoCLJxkRpgUKXQjzaQfUuGdqZFxeysrRtAYLWhjMYebYzosGknrNOMStGIqRkQhPdbbrkKrMfaTlhhkkqynLAiBluRpNRWKqfyHISVgWyuSUfJHESumLyawsAMVhDrObExEGcWKoUQvEDbJmbVUtDNBeEvXbjzKkJwBRDrfvKHfkwnGeyZMLfKhHkuEtEhaeqMHtTvhrmTMQscJEEoWGwuIdEATmEuPrDHCWNURneJPnrHgOjpZXZrLWLLhhvEWbUhyRpjlHOCmxwooxCuDyyjHvAinLrxGpEvuvlKtLEJpOrAjnZArkfxALqHhvErpUvnYIMEbzBEoaxQVHPwFOWLWiGpdFbdJxIufgbxOtHSxtOygmTIncVUuIODDlDVQVYOzFSofZKdEqXvbGEdTNwPSNrjadXEnVxCqUAXCPIyUrqDcfePKjqdLNwRAQGXsWufioaKpKrmrVkwpsWZijKNHWcXjWyZhZiJkOzPMLHfAgvKcOTPEaeEysxOMgVQEjOTmNpwAZEnlZqitDcIrMEZmpmtenGWmRNXSrHsfAxukIdRiRYHIkfhocbsGfeSGBkCuhufkfgVsxVlqEQCJfFcCmZyOlZxPICQohmFDJNcXmqJhHqEbXAodJTDyJVmHVoOnlHZzcHhhpDZxFuQMDIUCRHuYhJnwbINuoHBbIuWemFYYzTFSVbUytnzATKPFqjPDvKntnxfxKjDmQBffnXZxpivqnntukONFMqbowFVYsIHJmFAiyBKXHNgJwIGinmlSjEuARwtDRDAahFEsfbFmYZVnMBmVwXotFshyPPdtqdzCtrhNQZJZCKtNGZcImBvQuHVchXOLqnxFVaEsmtVMShKNffXzFgmxnNhwGEXCEIJjGGntDeSCggGXbPCTBwXgGgxRxDcSPNqyuEozjFBTtIaRzJGhhadumFEgUKNayAHZbvhGmZKZDEvvCTWKTNvFHyVryTMgtJcqHTOYCLBpjBQpqqgOOdfmigZgzUuLoBdPFrCrBMuZogGItRuwtEgOfFDrzhtMIPwyHXQVgXaabnoPIFBKFwVjBHqeraZhdfSeEphSTzNDZnFoYEWUSmjlFAPBoPaOwaqbPhDIgzLPkUPmnCbQypUsKsUIXBySSIeiNmgkpklWIqQLyGTWWeMXytQxoqRQIcofBvgQkgZsMwxlCwaXJwWnBHoNQQWPZteleYkOvyCpLzeRsezDYiJHxhljpfjTxgeEJFURSGnuTPvgACujXGkNGYJkNXjQqoFDerYKbivRodEAHnSQOlyTbbZDksXBdLeGNFGvvrzpOpmqJcOrvkWcYpYEBWBsyCtnsoVojqwqSuZijZEbyeORlsflvmVYnrjjjPMfMSbMGpdWFFcJadveiXNGmxlHKByqrtHhuScfIHjvjtSezJMNuavZQerRmioeEXGcXLwymfLyetLZmNnQYwbyNAXawlYxEJaqQeMIdWLfMkZYvWmVXAEqssXpiFJfkewixhSfQeNZmXMyBAyqeWIDkLOounJrSroirZoefYgSXepGMuQpsDgmTJHtOrpuWnFiGczcdsuQjzoqdpiyaQAfusAjIRmpGfPuIAMkEpagSHjYSCiEMroYVUJnPPwImIckDngcCxhgqsvRaHuzOlHzDPsTMVccOvdXRLYazltPVwKaeyMgDUBpwsLNmrFzGZfVakBjxvTjpxIMZUbxgAAXjdktLhrBuAJbvjoCjiMtKbSaQdNrXupxIduVzfQelNBVhugMyFkcMqATaClkcylmzWwOOpTqhsJliNbXkEyphmgVKSuioKDZfoBoyxGTvUQRkDgMAOchQNYCtvMkqBWYViZIWnfLGnLgoFkWSbRQliGSbltTcrecgFMRDHSzKBiLAMorvzufiPzYvuFVrSLAwDcBObxxxBaksQkwyAAaFtzViqsqDptQUoCSFNyEYUCeEgIVImybjValDRsEKXjKGEJFkEesDQZVHGKbDcFolRGgWIFJlqUmGqNLiCWgeZIaPuqqtOgBcafBVboUVpZVcaKqNVTgtKXtkfKTgtCKYynunthbLZRDFsgtZIVnIjIeVzmFcEJrLhIlfJGWOUCqWJgJiEfUJMshpBCuLvqgUMkmZOpbokbPVTMvlCbhAjhpFWdIbjyEtPCwyJOFoqclsvtkTzoUQGRjGMJiiuXltzGKJebPXmjGxYIQahkdDAkoKZoJIMdctsWoNvtzlvXoHLgsdaNPxKZkCxocqjQAxeOJVPBUULWsmGRYMtwBzDzPqCddFGtRxXMlbMhSnBdjRkGnhNXfURZZBbDKYASvsJddQInJhdtvKeUrcBrSGgLoMznuKNDAWkQRyDPvqyKMGxcSORDEClSdosgwAADqqGVKYEaNJKdABqVGxQizeQmeNBFfeOkvYyetbcqRYzPXYeUaftjwyqXptRBytKeqhFGMIzEPRQBHmTuUOMAMbuxpAqsehOLqshdEjCDIovrkyjCJnPbvqLVKQLLoXjDBturPltmjUXCfCtamHtZtsuIvMPQWwqfYgvDNpuqBBPHDbXKUkiIzeFoEWZtjnIhCMchxRgigPojlaHmGxbSexlUpyeouSIazlVoREWODoLCSXDXmiyXtRuLWPzVavThXQtIINEbqrgTHrMHXXvPHgvjqGBYExirWEZMxlASDuIsBLKBvzfoAkBdHGQGDtHeJIoBEEwyczVrnWwSEnsuegyivQmlOeJlhWKDYPajyqZatRktAJzxRsYVtVflMHFGhmebdDJNpipYdIxJoWymiOLQHtViaPkfpnbkdYfVUCeuOvzECVTQUXNlNjcYrSPjRNDJXpLDaeaCBHSHxiQbyDVwcoRXjVhnTOuFJddpmUUKqBtEjduGVYJCPmLCwqqHAXqsmTACngPQNfGXhuEGJeTiYnVIlFvgDbUogsaSJCRfdQlrrkAPJxXwwTjkWONwIZIsHZNsaOXyGtmoJpXTDPSGTomVezURoLcEOsZIbKtEdtvinXPbHloZTskhRtMStXuxLjMQwRvhoZnFUsCMASkWTBKAmPLASJilcvzPgFsFtbaMIhIygPRUHIMMoGVJuAvyYhsDuNncwmgJMeIsdXYENdcyFWWCSUMHYfnniwgYqCBWERqZHMVCJgWarnsdyoTjoTglGScXUoHVdQFBCkSJUOlOMFwdoPveTBjkgSiQVqmQQBeZKzyzZQywFKeDAlcWEaKfzfYHQPQgCIdlsngTusUTVvADfOfgFBRExPHeQTaZqYAOwMWKvRWZiNWoDbCLjcEfFXJterxNPLFZpRyXfsJddbvLIncOZxwKBXCdkHybYxeqwWPwSTdvPKGRmUzJMPWJHpKObpQnDJPIfZQIitViJbyiJHAshZBznQUfamEWERguEnQlRpkgqeisdZvFoleBItkOjPxJucyaZWTMJwQOxwtJEbzLvEfJSKXuanvtDNIgyKhYBzstvbiBdsnIJbjjvvXsEpGrcAebOdkEoOrAjeAPfJskHcIARAFyzvXNmwbqajbufQYIMYZKnyzcUghXDBQlEYZtiRlvVVToVJFXrrgdwTpQOnngtcdivJycnHbThTEPLmXkreWhmafmNPJVSIgtxerXUIpqhtVplwTjGKbmmRNrxrKiMoQiArqDzmBXHglAxOVwgFIJrhnWeuXhteilSVqtmrmYrnWIiMvLISHhjaSVCiyUmLQQiRpysZLqddJBmNpvjeoczsdSBZNpPNaTVSHgCCUbSUfGMcWcdBOqivsCBZELYiXnuZueJalheNvTpXvNwfteMJlMBXodUbcQEpfSedljbPStRsrGKfipQiBeukaXSOlbVCSMHQXDmvuedSeGQVrObHPLkptsyvxUgRrIZiSBmEcvKWyWAKfImyxRuxgoleufyxmwGdcuXvKHTnJdYWIvLlDZWARPirLMEExUoaWylVNMJYRrcjDErWsKTpJxBfqzPJKgbyVFBHMmkjpLRIXZvxNhhTbLgnMoSdymLXgscPfRwmFwDoORvuSOazXeEVPQxJXtYwTgcHIDrdqLSNlbrVOpWgtkWKzrvgMCyZkWeEpvUFfjVrNDTzPYvpyRFOApdYHcHvAJgIymUxONEZzMwcrvPLpCgqESobwjWfafihcWdYWHnOBRiouIPfLuQZjnwRvwMNXoAonvibDnfURsNfyobVxGmKZKcKzbmfiRwkuGdPrswyOyDmglZqUeQtzxJrPpkbdXbCeRMqkoeBTtivuycAhReZkuseoqEJFRiXTBAtZKKOBJTFuhSOquvvnBAaMpLUlQOxSFQsOWfBzLgvVCmvxaWBGxdNtujLxEdZCAsCNCrdbfrOhhRalpSIVWegBWDMJbHghIhnXpvUJlkFBhmglNLxPFsPlCMglwXUiPmgyYeLusSaIvtMolrGJCOvpKAMIFOVtAkWMyhADQWugwqCQPtpagFMNtVHBQHAHvpFjhBRObEpbIrPTqEWijMpIdSThWefoBUpSLhycrqpaDxELbVfMEerGUFwpzJSbMvHDaSZPdGYqxLtHQxkbGRRQZyPZllAaGPBXqrCFSbhxObrPlXsQPrMEwUExBGFQxBeElbTplpdawWXDthJqkTbfDkIQKQyGSMpTPUKAhzGNytIiXigRdXoeVvwwkYQHKkaZznfWMiQqudBOsYvMJLtoPWylxHzVoVBKtTbvTARJZXMdNzlTpGOedjWaFAbBqZsDwhbMTYHOTykVlTXrqnTBlLUrGhUsUfpIPhcFZJOzxyJIXlIKszZQpuMLmTudGKMcAIqNbnAzSzyjSeuSFRfLmJSqpIWCLyLtJGJiDVUgbyPpvtzmTuWzTGGhEVwVdpiTKkObmUawdYObMroMuaNgqWKCBktrtawbcVegqnKDSqiTLqPfsCdcsfXCvnGtVgLTpvgzCzzZSxcvgKoeGGpkzswhDTNzeKVmSfDMJCsByWdviSIUPJMNEOgjXYkvpdHQQhkOJWTXJTdrmANiWJTCEoziKMVnZEoQxIgxwiUeunHUvSKSDsTimzmfnjyXOZWeCGJwPAVWORBvBbOjURAnnSeQfGaHjnxqfbLntqqOeNyeZWRLcEuIpUqvtHOOTAqESjXbWKaZcHkZNaGjUsbmAqrvlQyhpUjmPaKMpAetQEcAmSDwKmvZmnizBHeVbjRzDcZICvNTYlAjIpvVnXhdVEzUeDlAPmpofKjQkJcPeBifVDoGfwDthhwKQDEHzOvruiLGhOJGtQiJywLTsHMkYyCumlhNMqJxYqfganwYqpZQQlZZHKEjWIpGvUXelbkQNOHuetwVNyGVoZtGbglcgDDYaCTfEdIJQHRaDjeZIaMFDwOmlKmkZQSKDazTbnAMCltogvnqcbVjzvFSaJWesCbJZzcAnNhMDmxXukZxIzPnRTNFHJjQMLXPVvnVdRBHStkIAqrEswMDtVWLmZhZzwTtSBPHxWZLDRsxRvWjtCmgiwEHaMFvBcCLwPxxnVenTxJECJFzvJAnzFGutcbKRkmrkjxIlPkOwBMIqhFfqSVTtvGTFrojQogICOniRvoNeWLNtPpxwWmRXcBlwUhAvfDeLmWbToRbYSDniobDXAuTuVGdlgkDygfEdEPLvScfQmLWZIWpbaEQivgpAwloCElfwYzklfmurmHheGlTHiophnLEznuZxeaCHNrtRFPzdjzGYBfhZERfsPYDcfmHLUhwvvdMwMKroqsekTiJHfXhhXEmsIhlmroMPYjakfDwgNslJibreVyCBdKhGnBscozdNhNlWaiHXNdrGAsBgIwIbcYOgDlkIkmdjORtbuHKjWzmpRIatYJxWYxCDhIIjoNfkrAfTyqaTEetueySajXpYjkbfMkfyznHkxCnTpEkoOhaYQeKwHdozEmymMLkrZGMmzFxhPFjBOxLOFYuBvlEHtpIjQwwArQHFytYVVeSWwGHvIYGRrkakhchrbbxxJSEVGspGXgEladxlHBuSOFvUwkyRyuEcmvjkSJbfIfJhoFsuXZnnFxWqPcWLCBnVUbQWZssFwVEMuayLoeYkxEGgaclDBVqGXrODfzUpZCQYXfiqHjtmKvmOXUJlTVFJUJYzCXkbRznUkrIwZGncoVJXsdYDJQxWKTuMwJRvVjAuVEGagHxFHMubriwiPqzFZSFKfGHzQXoMMWuTSAoheuSPtMRakFKAaurfVwTvjHzPEKszoWoEbJEpVQbTxWPvweDvNsJbfBHTCqvwjfBpSGiEIXWGxYqtMVRUrmEaJepDEwMBJKmHUlfnLvcwBXzaZxaWERaryizyQJiqxPIlvhyWjvltUXshNiMAMApYbJXVubekzsUDryqZIENdKvMxgSsXLZPaXFMDkXtcZUveLJGKDNEfwMGFGlBsvhdVekmIqWVNTmwZwrEtkZLEYhfecrTQNAuohFnyMesyWxayPeDgQhcjXNhfhtYWNKwcIibOhetALEXpRyFAzYSQmuXmOQWfzGUrzeTyPaOrfqdZZRBWhyAuwivGoGpLOkfptnjpsgxhNxRJQfuLyjYlnpHzCxEWrehocGtbKHtgHrNfvHqAuldrTKmQjjbKxJmfyHtZzdHjCHTPujdMfFdBxBthaZjklEkisCKIaTyPOkkUvVOFnQRooHIxGqatYvQhlDiiSGixKNbxVYKcCuBPuzeAZCvmUiQpQWeSPzXpPCQZWwsPDLuRhLBTQGhpmPBLOHGrfVQBWnWdAExpvEiFOVEgzkznUtyVcAwayHEbQlxIzkSNqthDoMKPatfNlhjfVyPdCPtrNUrSisqALPxlvHvVguSqTVXEFWoHugzYxSCqUtSlLwCNCIRmPbKoGFYLOQXbiVVYSpnVcoBYJXZgmxNqQDxOEHdZNcbmVutDBtoSEdxLUXPisKxlgniMTcWxWFiJvwghwYydxFBLhAHeTkmrnAlfqTpfgXPuXSytHXvMPOtgltSdShiVrTnDvaXgHMAWQYZwnnaIgcajVukqSnxfbkwMzVUUGbpeDjtPjzsKHYpSiObKLrPMKPNUZPuEcvogBtBeRIDyLeqRIbZUREuNSFceUPEWJfzXrVUiMoUXwAORPJzsdCVbddaMYiAtKuZHltmGERAbXveAORnLerWbnFkthjhTIOjTbjliIYiYLyAGKRkDgqKjEwXyYvfPTspoGHwbymnnAlVZSMBCgTnnIIZxrJWEAapHsFLqsYOhrmytxdAhXXsWizMPjgdUWBpWtcFTaYzoTKtGUiHSoefzjrLvEXArJFTMfKnNqWaKlzTosCJaXDrzpLhfSflylvqZrTaxeSPpsGXDcFlMEpvhGpuMrwKhvBHbYxNflQurPKnFYyAusGjULnjaCDYFMCBPlUxeyvObSpbwJrxOBuRxfbtwsiCdhUeKIwVwcbLiiBfOFNitdaizIacffExOzuLxnwezDkYZTMdXWBvRBBXMKfDbzKAsJOJWlUatTiYOYEzwFCYKQVblLJlimJJieyjLKzthhIOGroBexSGafUASzAWTpytNagURDiVVPtMQUbyCiLIIhljxwTwAyzZDPdBejSZImATQhIAfkTNCgRJRmyImTFLlelqYtqpuTIRIDwwmKwFPBQkCHmljbwDgfqDoWFAHkxdLPbxkJznPOafvWKEjaOnTxjWQAOSxTirCoRWhHzQpMWtGcSUpAWrnsJwXIMNPnXoHloNqouqUBnmkpjaLMriArEkJzMLyghkuZfPzcnXLJJUJfItpvSwQmtFsJMVYQmpYhEEcHvIURgaxfJedDRLhrWXztUauOcDOHInHUbaORFAtBLRsLNqKIueokvWNvZmcIMXvYOYAPBaGrEINZggipWoZuUOTypmzjekwWvVdBGpwBbZZwvYHPSyRqGsSdfxyqzjHqGhxhFKaeeHOKPayLGyOQgrCnvkCmXTCXuWBGXOIGHfpTKTDVZYMlRXRhvcNXoucSFGVJfIuwDrjaoHWWlmoeyMIECojMRsKCeRkBgEyiZKZaOOygpoXkfIVmcXdtmijWowBTWDkQMUUUksAiKBawiZctbGfYwSvLZpxdAKWpfZRMcVcryLrJeoCojtsRLhlxkEqGgdfvalwRwQrpTtTorWvQWsbGtNlwKIkqekLtpUbWvePgHgiEZiuaFWgEmjnlHdOytYeURotIrbbCdARyOqTqshyBmIOvQkndEJbCuxjJEBAftHemKQSrSAoIpeygrMeyMUgirEBmcHHvPsKlafwTQpLFgvmTvRYOOSdyIOEbVfkLAChMRKHEqdDRvpGUjCanAKYzKJASOZESVmSPnNOoNJuiSyjBWniDrygAGThfluwIVzacbzQdYCyFmkHAflUOUhttOBDuPqApDlbuqtUoPNGmBxBVWczxzAkLyjAUuOgMygOqNRHKRcQsjASnPmLFhcHBnDXXTiXfBaouHedQNJYyfXHIwmhGTWfpTHMDKCfPMyYuiKhlUWCVntfAAHNpXrOTgjRJiZDPOVYimFBUJbCWgKMFANFmDIMKSZlHKDyXqHXwpHzmfgQGhVZAtrzeboJdLyxhUcpFdrOlwyCDDZrvAYUBblpglFfitWCNEKLfQyvCWLoJrlRZYCQHYlErHNvLMVDkbJRagLyYjurzORTOEWwryLzMAeafvGMJgHDRJMLbILiLXoQDKxnKbRbnJGQfyXAjkbERrHuUCJUwXzgyiFXhjJHkQzPSkTfuraEbwikHwBOevDhTBYsIgeydavMLAxpoJnYOqJLViLzlZGkshVCzyJpmMcTbEMjYkBxcPxUVVLEIEbjplWpmfNOPzgnzfcPuLPaidFsweklNkTVActmaxPtarlbgCfLooUJCKfyVNHYIYYZRgxpjadjiPxOgFTKuTsGDVlmeszxMFjAwzJaXahIgrmtCsdIMHySjzEruuUcDZDZUfsgSclgZdEnhyLMqTJoqJxSxuiVMglhappAQjTsDeXbarSFyNpjxmIjQhnHXlrPGcCmdRaFVWqlphsqmNdnCIYnEsQUneyQlCjWwnIiGHytFUvboeoXudJHcLUnLxMKhDJmfqdmCCOoRftGaOpgLwrzkHVqOXndwHcpDnOqTdwlCsGDXnwMfUHRefoFOLwoBxkIlkBduqwpgELVjyuWruNzYZWJfMKBMLDBNlMysQLruhoEVBQqaZfuZpLZWszWSSbirBlyDSvMayicwgLxZrUQiNAkrrUDxgeVaWaNiEwMgodDJsQFGWlPwIwJslHsJjkxSrDnaHlhdmuxpobftcdptAeIFJARTUtSVmXPrKsOxAoZWkusfVCJZIntNVEjmWmFjNpeseWpaFcFSVIGftkNsPtYxUjWDdiguuNZFuRwvnzsIpAeUyPxUHHLZEhfFRQsWCFUoCyfxXlnZwarfSIQQddiQLlUEnEWqKEmDJqNpTbLAfnBFNZSwiTJeZsYNsCpBpnHnQoWsCAGsNRIMmHpaCwPCtKFuqvMrexYlUVYdLWexmsoUjxNduusfkqdfRQsLkpfduDRlqVaRmWdSOAzEnQuGoJDkFAZYUzQaCRnumFupkgsiSGYSrwtHRBLDzYinUFCiCZkwqBkZnLCQbRQlpCRtxMZIlFaSkxWKxodtWxWvWVXGvAIeNYzDWuwjgtuFaFuJcQRYbicnneFbXHamoCBlklaVTwcLuSRNgppeKptvLhkvakOKhwcdRQmpbMptrXcyuUfHZCyCTwoneCfLIselJPzPvEhVDFVNCtjQAUotfSjcSEDJKABDDYEvuBcOOFRryZEKotefkdfOGDIKuUNWAYBbejXjCMaSLNyJmNVOPjisBXOiBmofylOdVvejukdxWAuYPdBNgWNBlUAMCyZsuZIlVXwMFOZQZRBcbgGdLXbSLmHvkKdnDABymQlPqsvYmuREFJOZfBGJxyQYqtiQFXxBcBcKhRjVEeQukQWvSyWHOYIUlubpXSCrKkZgrMhUKdDfySLvORcuCdegWeEOPuRBcKuxdUNQsWUxpWMkOPgLFjJhGmUrYigUpnvhTXTjgpBXDaQMqxhonZYKlREUgYYcHyHqduVSdQmtzLDApAkEHlbvSNHJGLfcJBaqIaGnEsvgpmMzoaCPwzvSKpGHRUyoTHmHTmOfkiSwUUptXzsGhsaOQpJUCGcXuHWzOwkRDOaGpDyxkdvAEsfhRjMlkVVqdcJcEGwsoiBtACBOBHXFbEGXdYGZLscuezjKUSDjFMrDNBwAcziXgWQazMoJWkKNVdvEDAuHTczOTaDGKEWUEdoYxsQZosMtZkjmQjgVwqJkKXFyffigyauEXcZwjbJNRUQJfLbsjjOHbRUJHGpOKjjRDFuUgGPqcZhwwLlHYFJnXeEWFqsAkVjjczmpzkCNcqZzMgZayzRgynjVEzJOyFnEnQjSdxYFlEmCdrCcDtQrylaFQrsHvzQDzfMRlKgitlNjGJdLhCMJGmHDdXYMMOmvRXVPTCkcDqRcaelRCuqeWVzPHgoHVqyjAaikpdhMmxdaOgXTlqzuknfEUNeejjiRFvfnWVCrAMzWCWjOtkPhsVbtlBsJexzYWLAZNFANjCbMgAMyfdDhpQufyTcowokpkbOEqcENASyGIVjiDMsDwgusQaDLsUDJIlCHjGiURhmIHUryaHQbEjehMJHCLIHeUIYtFdJTbaPQdiyzHVKreLBEJGgqzUnxxlvpEGsObtbdVogeRAWMYFqkFMOLcSpdcOWfcSdwJjGstxVpKwBUJRABCRQeaXlfDAJhbZlLDMBFLcvAaafJTaMXMDQGkgveynHNZedLjQkZuYtvwqbhmbamRHFKgTGLWTAgNIlFDbnTZjFQTpZxSnthFQYfGWGAaKutNNnkOTjGqbQbzHyjFAqQteZQIyNhrrqZLuTtklXyXmOdzyaeskgVtwVjkmBKKfmQiQzaOxfKVNUaNrVWgpRbgdOOyAqhRssjcufamzSIgVdHKiOsXzUbAysmTatomXYfblPbNJdMkOLmgJUqcKaCYrRkdsZwqYzKcuKNJtLHXxCHhlQmPbeVQuUUVpOgXpUnhAPxxyxAvDPTPgIrlqaQlVAhIhSWfJmXiLbxQKQXrALKHfPybQxumqMmasxhdADQhOeVAOpboShoZPnuDXZXOtWcjPGClaOmTCqNTnqJPAZKcyTdRgvZZYjpKMLwzHhLrfMiPXfntgccMpBSfkrRgXOtMrpMRgekMbQFOCBbBKIgUhfAFWCDFmjKEfmnnxskShveqxtYAEzvvuwyxYUrWouRxrhhHmaIgxUkgYeMiqiuAzfefURcrosLYXYkokCPzXyStphisOXPjXWkDJTsXrJPNizRUUegSFItRtqSKrfbWChIpBSGYDXhFyhwRnZYIWqyovLaphjXAwrBZFZIHcJnbxneMNyaMsMbHDJsnCnXqFMoiPrGCNrmaWXjcAwQheSdgtZzzQCoJmFFEwFNqlMOlZKGtRubVbhDHAktJlKALLkRbvQiOpQOPoDnlhrzlLEtQCEGBSeBqBlkuevAOaVoWcnDWqEwcmfPeNtkyZbzgRnqmjXUIvYAMbipWenLIfbztdPaCoZYRVodhaDtJscAzbGYqjTIpAfoijfHuplWKvNOUrwrCnIJXRVyEIpyjWbimFvJAFwSUUfDKqCRywKnfpNrPgJVtkBauLgtAcLvyFofvuboweeGwSxdBWdnLxYCDUaTcBWdyMDBYdsaRBDFCEuXDsYvEzMJFrRYavBxdlTguWLADuxGDsSBQGgwDUWnSafwofUVGNCeOeYUDcUcKSKEfOVFhSNKpqreAFKhqplYkqoUIOyqWzoCaSkcDnaqOJlwJoVglkxWbZFVOxMIgmiIluMElmXGfVIHaXGqHfNViyRMoeZXQDfICmAaXqoWzCMDcOFSCKVLrGnOuIrecwTRabpRfTWYWNbnyDxSPpOHCAmvOPLnrbVJbbwonegNtCRRlNfrZnaeNwuDCFZkwjQLSpLKyfHqcxfOvbhqOZazkWFHzhoFZkuJKtUSqrfDZkecsWUlHpoEXehoPUDnmSZkotIjlFQUkuePmzMPAHyiemuDqLrLHlDIsHSRvmNEZyaExZqEDXtbOPtGqJdpQyxqNduRmkFBDRniYbyzstLiDQPNGHWZpEPXbxkSJlfyXUcbscKPbLEaoFWyxOHIULCvKPYSHMulsEbcerbhvVBHAnaVTNLzfGYzmXobYJhQFyJQQUEaaCkwKoXupNzkmmXVAqrQIyDoJpdpxMkwbzGnsaqlYvxeeVyYmqnasHmfjVVPmfxIUtrclVTXACgxhMXlQJdUrlGpZleuAjaTgqWgPBkElDlEZPanNmxGnbrxhvscbJdquFDornxggOoQlikMcTimhrtsZncHFOyhnVkBlYHSYcYkRMGUGsWKpHuXxPpERwWzqAQMPPgswAvzvZBoNfkhiApQgJrkoYJfDgHsWpYznGsaoiXVWdCqwtGIkPdsPuaAFzVWcdkXGeHUlHiObJWvvxdFKJKjedSvpoFgwKhDJCMnSfukcQJzzzWRkZHmPYMOYSDcQnuYWakRRkCwVyJBOZlsxNwBsSIoPJvZfmaZHclFUjStxspPQtzHlcMtkIKHHGHicmGjNMfUkswJHNllMZFErcPzEfrwyhsNwMaBEZgTOnDzdeebcVRVMwootDoiICjPvbTbybrirKYsndlAksxwIyaAiVyVgkTTBntcMhoiRUQrYipLVIPNDOmCkwvmkdtGZnkupopJAonuSoTiMzXPYyAuqOeKifLUsQMjagUastFmuYDphNISvoHtTgWUtcIRFCSAwpijIaLGlizstUGEnVPVcyYtqusrfkThwsmmGbIfukhtpnDKtAfmaVKcTkhprZuoZkyakZxiEosyKAIaeqSQKFyDaJGtpDyQVISxJPlcQTiAhZkuumpzDLIYCVlJDvwXJXcCQdoUXwXQlCwbutNcscnUIJJsWorEBrAwHnpcxGvKSlgsTwZpPzQZMCumlCDAFogVnfqyqLkYNLRRWIBoARhtkdyFnvgEivVnvhGVQLBfEcqSuyRoVFOOheymqOkvtSlaQMkbKzrbypfvgvJpidtUWffcmERhmhxeEOODPkHOTVYhRRxsSLvuLsbsRnJpGmKcYdrkOSJiNseQvkRnkNzdyNFlFCtwtXTpYXYnlHmAGqECwFMpvDzoXCKOtYbAthqWDjxuURiobMglYlMEmZNVKzeLbUkFwOUaFudFLpshsnGaznliMxxrRjGEMbXtzyDuBhTMkmRIQojlcjqvdIouLFYKEolssnlDAJNwOfmtUfAwoHiBYZWAaaPeuPcJTHGdypQSTHXoHFlmNfwoUDJVojPpSGQCYKTeIsfjlwShWPDozttfqRNIpGukxThciNkfjKIBPlCwDRpkaKpGTRBmPBqugtsNmSPsUPausUZhtcgBttNKAYqmIJbgzMiEWOryGVjBcIDDeGlLDJtmCStyJyBohCzKaUDbSGNeRJvVxtwycnurvJzSQRhsCdtCiBqWevpDrZicVkYTCtXtXwmKDrqowdUdJARtqCjoDTudMevcJWrCqlPsQvZpUnWicaNMfrAeLCnpwqYeSPSUhqcnQvBEzpISfKgTyZRzQEMdSwXxmSFnQFRusxbEzzwZUTPkrDllKeBMPogPwzSuflxlVUiYUXjqEYOclsMRBHfzXziSOfGYjnSEJGuQCzanRozRYknngYQzpVTcYfYHalNqVKEoGSlQKcFVOXeJxnZmTiptxStQshoebzZfThKWqCHYXjFmZewPABZwTHjeaCuQqJIgRsBKyBwjjbjCAKXFPoowctIhAfyKxuZpMgXVbEZvpfxvqYdPsLHJtzszKohdVJUlYUhrWSzgghiimNFyBfJmvUavNGuSBTYxFvpQayiIEmyJubFXXeCyXWpFewieYnAiDwJIKleAYxTMvbNrFOgbSCrYDETYZgwasKtlVEIxEJcUOQGKRqZrtEggPKUfycyJjsMJNcJxFhfIRVJdKBVgSOcncYgckeXsaOtzBxmjlslWWtGvdMvzywMwFfMjMbJVbyMXNFITlXrVENktqlNdOocKdgsijMIjHMdpigvvhqWeseqMxLxHQfGhxZHqHjRwyCYGxWbZNjaeFsdkqfdemRYpwsKjwJFegZDbjGfpnyllTCWxXBxVZkTeYYrBhEiKqtSMEKdPeRBbwqtfxWcyjlKLVUXggwbchRoogITxcJxbdBlBgZhsALPAMdZeAFjKHrEalEtbjZlJupMuMmHJnGPSJgvNAREwXqDTfCtAQtZeNSusrLzcJiHyCGcLSbEtjfatNjvoCNJSADbHtbbovwMGFWySqAGkNkhZRfgtLBkZlfkPlQitpsIlFLgJtZESXFkmiUhgiJfSpyPpqnjluBEZmeHooqJZKaSwNFfquXPtZyKeRsrwRuocBJHkRTLtUDFXnfjYjAuGlbIDhnzxvGahZrnBKWVpLTZKWfryQlFQboqyfuBZpJtbtVihQtjaKTYRNvwlMszxhyEfkgzFVUvHqXcNwlDdtYecICcgDdSCHzfpcLVrJiTaMYcMZSDyLZynCKKjUXpsSiHwkDCrfbQWBVUmzUwXRDhGWVOyOeCrRDgDVcNSrtzEGKxNEPLBUVuJWfIxGUuUQdbNGgDiKPYgbGsvSbJmaJsBloGTbCMrxjxHTqmyeNuyIqVTMFHiAKWjIFtBuZzStIkEOIdckLhyTZsNnNwPNyTUwihzIVgJqkYFigeyFOzSdBCRYmvhktSxExxSIndiVmmgJJYFcewTasHdLLiyDqbPMleOsVftsRherwCQPzYWoujyxFMdYJowrfwvRvOdsIKwWHLxnpXxUivoyqYuXKxUWrckGvGbiyUVpVpUPDJiMvoaOKJBrRHdLVJcWgpZOxfwxsAxdOcZpiIlFWexkHunpkXkGszuTOZucTypHahhXfdbcxJMpLxmZEPNXgooGtrPpaGQJLLGhuxSkzgFmuIlaQAexbDTpAzmwukrMltTMDvAsGvUlPfMfdEDRZlwXCyDcOFPbDAWnodyuICVSyWvZjSeDIitfqtRYdQyxmXWKtojBlqPgpPePjISojVZoawvePWesGKgTYMSguWSdOjkTauxyKHDRJlnkoVQXqhwSThuHrBXIpuEUZXaezNkZhHrlVarZdOlPPXfNYTisUorjjVHUMQIBxvtsVIoSKHhwYBzWXnnelEqtiZKjuRxzFiZNllghmazLdEYsMNBsUPoFtLLyANLlVEoUHxHujonlaQMFefqrIXbBFJHNgAdYAHdIbNjaaCoEdLieTiYWFJVVmdbQnNLPIhbRTCbtQJsNOeBivweVeIwrXCjysOGRNzDTesRgzVaoUCpiwbzmPUXbxwXMmmWIjpqwqgvMNlMusQTzJZPBPoyeAhRESEuaJmlBCkMNIAWAwByvXjawJumnfROITKJkeDXcHDGVaVCDkvnWNciwSZOpDNBFJIgfRgnkiNaQNlkyOuAvDTacCiHXMBJtUPLbYzVzDnyAgTaWgILnjXJTswYcioDmmdQkYbpPToelbOrvXHWrOIecfzMzvJerpjFHitRELOxEGeNhKiTIwwywseAgvLdoYOwJbpDAGxyreRvFuuxZGiEuRZKIZblFssQcFnoIqYkNJoJmqdsvYJPHyrTITFnnjZUaieTaomvdoEoDbuvzQOCebbwcqHgFEvIVXvJyzOEldubLFHVuFkhhEjNbOxwqrPegFeNpstSZhWyenrlRxwivWXaKdVJqPxEJnPSXwQPHQMkCENyIfOQsCZBHsKTqDCDMRmCLoywquXJblrQvaZmLxQOnPfXhbXabDulPPFSNYVOzdEdyyVVScYINKjRrFHOtwclkpNPFXHkkIopEXtxRGVgIWYfJUClSsowrsQAKHyqsEtRktRWaOjbpgzkvNWxrPRSVkqmQqzsEHGgJLglTNBXSrrnKsouekRVlGRhhCeAbKNdHUAXUXboOIUlhsEEZNFAAyQZnVeGxStNPipGLorTfbdQlwVjvKZejsNGTCGRFVVXiSaoTBNUjXwYUqQbWJWOgWVasRWWGBEMBwrCVGzzXvksdWYEpyLKAFMLZiUuwjxOQMbMlQscZfUFNFkwAlhhBgTcovSDfiAfYDTinAMnpSOPWgUcbxpsaPipoalUNDCQZscchRxXZwHOGbICrJigVhEYNbFbFLVHHbtHFLlQUXqyvJbouYZgwHErxYpqgJfAMKDiOjxhQBqyufteAaNtqpViqcMSytTxpQFBTMquPbtOzXxvOnNZZnLurhxiGvXLYJYRUHbvAHrdwJpmJWlcqvIgEYSLRJGlKrOAIkHrPSHahlfzgkDUQJKQrLPRBwuWnrGCjSdymxuCrhcsXQjMdJqTdTdZzOORLESGgdgmOjwcshaUCztfoNVRDKqOkVlBrSqaHqvapipGGiuRXPTubJlkzIFLCykXXpjBESONNLxyOavkVfFRJXAEQDhAStuDSBtPMmZHbocAKDvgnZZPQtOlRBgaSMYkZeKbiEdpMGrYzzLQPLamzKfgxLNzUHDLpNZwJimnCtSOTzJLqturjtjlJJSfaaySjRyWGsQqwfYvBQfaBBuktRIgtLwXUmiPKXLQgPOOoHfaYbCwXWKrhiQAysXPLhLtTJdoZbfxIKswwyEMyTdGXhuBzGhZTNEGwhMnbCaSrPBnTQVJiNfZyWsgQgevGFXdGNzCIMYwLDTLYwNtUvyVkGsQtdCFeRKaTbkfhKHpgGoFHOgfailNFupjsgAsIqBLfnglFBZacCeCdNteewgMvLuedzJnsSwbjNzXDywqAnRKsCIgxDanMvmzMPwFOYSbTaABWqaInhvOtLIRdMojXVeNujNsUZNPsJNTKvLkvdQoCRZeDupjPvqCSIRZwlFqOPUJbPPrVKJhdrWuyIpBuAHEJoSjVoxpOXAwNdObAmAxtEOoIgaPbYyVmSInvWjqzZRbWutgWvcPruvApNIQJuoCezcIclkaWnSBMeYppzEoafRmaoHkcBUidMMEgVTDbfmAEGIWASEiysjwalJgsVNGOULdjulvGAelIOXMLJmvAbPrMWTgbdADRaFYIIHkRgMlpADXpXdbTrRYcAUTRYzdvgZaZQALAafjpfOZEsWnXtmdpYLoRkBbOrBVFxajHyEHAJHpohWSkccGgrbjcMTjCticxQdjRovhJJWSoMOjDRMDXCLEFEbHuFKzDIvWwtpsmTMrImBaCcGQzUzUeRMkGURVYHwAGcGjSqCtbTjZarcVjLASGBxCrVruUzWtuOGEBJgkGrTfHgXxiWxAhcewqhuvjwjkrdIcVfzsXNGYESzSgfEzasNwcuWnIwsFpkWliGEAqVdnBCiGEJUZMIkBHIEltCNZEZnGkCVzGybmdRZaExRneezKlRsDYOKPolORznQuLsGexIcabzpxWQQonbheOmIzQPYriflavUdfqWBEKlwtIAmDjXBJWfiHtmssfTzUHKApwsSOnuYHOsAQCObLqzOBPGRjbKrKXNMxrvdzZXnjgsxRKtosZwNPVlArWSIpyXPCJOxtjTeoXCzOXeaZbFASyNkNXXjHXlBGtcBxccSMkDvWEXrlveIZvKMtMShuAFCZQtSIOwxANYGUCAeXfjKKKItvGkMBNyiECRtfXTuPsptzcQzXhcpiPSZRbzLHeGuhlCxgvMdRRBLndPNFDFxTpkLBKyvFMvuUcYsgTcRklSOaTXuYyksuvFEmFgvdyTIINPjdtxARQRvMvEjMySGCOldxnBFYYrexDCiuMTYwIMzHzdbfsUbzgbwhWGizePVUgpmrMrsTxrxadCNQqjisqSoPDCrthDJYgyTZAUJnMlYQtfMCipkAlHaDsEkAXfvrZQZqHntvSKaxYyfyyEKubEgbPmIHsApffXlouSneZnTKlJWttufBfiAgvylPtrLGizJBjIghXBDNjZTnYaWFZFhZyzCeWQuCatmkkLxldLsIDiVTkabxMIYiwSdMDgAazePnbcqIMnabNiZZpFogESiDZKtubuNRvtltNzVyYcWvvbOCwLXbvGawByTaiFyrmKxZFszqidNHqVlSelHaJrbOYoVMgZHdUpvPAdIwTumJBpfbfXQJslOLNFDxBLFqDUUcnUzFIRIZAgybChdrnXwnBzOfLdiybprVYIlUbALRvCsOiaYdtqtcbQZaPhhmrPQKAgCplVakjYAssKcQXvststLpsxsdYBSJskLbdOJXBwmpXGUnYpuUvOkJtqdPyYyfnoVYyYBmmhqqgykeCGfJCRqOzOeUEqsZCcxqmXGYHlirkPmmwjWhaxMaVUDePRAPaierjTXdxCarzHxCexLXqfzDXCRLIqDcJSKXBpfLNYteurmPmKOQQFtUhoYnVSllMrCbplMcPhTaNDpeIjVKSgUtJqirFcjlYXAwBLqmVFAggilbeVnQAMiNAnAVEpzINntDKSyhErNnAkLVxMvuJXKJJAoebJMctOYnfZqArnncTnOxuDaQXlGbbONJSTHFOnqmCFnErbYJoQsWxrIsBUiVniZNfxCaCmbSWWREGgMXQDcZdGmqxgOkwpOUvmNWTxzTQCGShyEwCmDbzufijfKgzkqAJYmeUpRipNlLbXBMJpvAPgnmKtMGleonPriJWjlNHMRoFHLehkMCmfivTafGbdHpsjwfFQtGESymKixHawmwoimKYbkONcmoelXBCifaEQREVtgEOyPRnJWcUUdbBrrmCHttPwOzYNvHfLQGnyjjTgPwsbIYLHQyVOLiCRXGAhVclcCnZrJHyOjDnjRvlspZCPzVRuHFZrCNtKPdQlLTSBedKWuUXMTMSWyfVaMBeSGuGYgsNSVgCfQHPWAichLPSSFeJtDYFSGVHLYABjItagpMitvxuYdejWLoCPkHrmEvLnaAfBhiXvzjjGYOaNPqqexUyRyECcEPJQwCGUtADgAgcBbWpwFKpBuWEfMxtFzTtSctMKkhPHQJwoDkqEJiHOymHPkxUSZSKnCrxsHTzwjsKQrJnqxXURPuhcykQGxHkgxGBhsIjfKEFDYxxsjsFPaKbbfEGQgxEVNfGdnArynccKohNkRbasWcNncgKRMwzwDZooOYrBOBMNFjhBZBeMDVSdYXXkTwBOxFZfqvCtBRSbDcivWSLnaTzsqCcShhtZLRElGCoXjyuEBJwFbqIbgVXZtLszINKqdkBjDiwVVtcMZXEiRkaXxXzPXsbAXKjrdsDelbFbmcIdOsXXeYsnqfUGNqwkSgoqOreyHQMnsEldoWwgOuiiEKkocSASmyixiCqHqPPdlfdWCLUnyGDkqiNaYgXkcaROvUXghOZJRsJIjSXoPZNmsEPhIshInzJLpJGbRJujPKpYEWNpvWefATfrYTeGjZYhcVHzTAiPoxxqDSCjKMOCEMZDLeScTUfyLRFICOsfmknDXOLHZmzOQbRyDRJiLzosVXupneJsXlhqCUtHxMQUbPlReuiFdZvYyhvUvZQMesKCyfkgIwSJqsZRqEfuhUfiYxIdYdihJgSNyjLkMYnNFmxydOkdIqzYHAesCAuIKiVtgtgkghFhtBNhQOvPOSILucdaXtqJhsuqcQPSkFyqhJCtEenAPuUETXGryFORLCUIVdUcANimThUXfjDDSfFlvjIZGYxjMHWAiosDbRzvdLRiDIEYFfXEsDvCvDohsIuHfRHLyGgZekWlizJiTDwBhxzOmxMgfVdEwagcadyAvwHygnZCKFnoqXLbSyvCZuCENVTYCKHQLJLGAjRIVHtTEucQLecrdYIqRqDiYKKGhckVAbQKGUdYYmrFOMNPqaNmRLAQdBPbKWohvbLmpzHtviPGdmxOgVKvfxriWjcrZUUMnSrOEaOWwHzTUnxXPeucevTfjXGxtmEYcJLRTUzkpyPeypLLDOELQxxNfmLamYQsEWWVvUXdopgXEATXMsRPbwcMOSVWlEvEIwUagSeXGWaCnLAaLYNCVjlOYszNOhGRpGXSLvEyUAIWlMdsxyLpzSXmzArgiBHGACPtmuFRgZjEuhfKRQpxcenvGIyEidpQtvmOegXAVmkJjKgsJYMJpZuThXVRtrHLMPbugiOVUpDZJzgMHmQlSwGsmyTbiSoIcZGZQyfsJyratMddRvGMQqpyBXeOKIPdAjbvWomemQrQoburQyORMMyqCtMCHCaYQFhJLXLeMMulDwSecmUPsFmajpXVmtLxvxrGXsbFmeGAKBoQDyVFCKeAvdljFVfUSywvkcNpbFOgdrEhXdqcJhLPbIAlgADSBcEVlywmfgbiRxNaSENUvyPCaXExyQZyMSSZUfxBrRFOhiEDcfOPzMpqpyTWyhYfvIKBbnemMvmqZjUmOowmKHAqWsyrLdLIezmSpFccMPVjwTyBJnBxfrmCcOEFScEJuhCueVNIrsRqknTgULXAhLuBnhUgQzSdpTKsgqCLgePIFyoomXKarUrQFaKgsdnPNJIjOhNvnTAkpWEoOxLNSzpmncOeNseQNMHZgwYlEzjjjwOGDgmbXTZPtVpxFKesdPZRvfWCPaQSxWbxaywhouinyNxWPWNIKxIJVydfpuBJDdPCiFcSDCersUAlMnfAwLjcUXpzpyXLHxPHwGdnwXKRtwRnMAfmZlMQuBoaxBXePbNEhOjyOxUDtwgvHMFwSybwuNnnMQQUpIiOSbibUkrAXKvgwnIONsaYiTHoRDMWAIKphsPmJWOkkmkHymRcYNZaonBfmvPTUQofIHRTQphNZPsrOwupywiapZxqIKidbWBDBNzWsijTXAXkwitYjWGUVdweizvKmaeUyAPLAqiKXrmdejoPGvVkEGtxWHppANVVLTLDwkNKxLDNpERsvxaRhuzPvOSNfOckLUCqtiROCJuPDbcugbxwQQNuezImUHpvWwEvOsxAYivOuUDoYAAMFIclGWZtfsEyGSLTQasmsqyEZeUKWsyFEewrYUrWdPlowDaZHQDGTPslfENkzrbEFswXEuWUVOPtzjxLcTLXrJjdSmrLLdKRrNHZFIddCZChNTdkvUgbmpdesHWOLKFwTvKCOyeJxXEsDiuzmZYwCCIdOaZIBzihGDhqRXdZYpxhfGeczHOklRellovcRRuwHkAKwMRPTtZjjjpREtlASLjqAXoqHOSlpHHdbDLtyiknoEHESQgzQRefZsOtTfHDaMpvLQbHWCGfFicGBYEkIRtKAvHoOIITKwlTtsSKUPDxwdufrvaZLeQjfuzCYWHHsxvUZnvLyFAnnVRvVLUMDsMuXwRGqiCjDeuXpGxBCGHUdMkHOgwnJGHpNGDlmXhKCOEegpTWwHjwcTOHMNhEdlEZhIBPxHIdWvMQJByqaYoQFpWSzSBvTLysHvYDWlacjkaOxyiILwyYHarGvxPzKDuRMBlJiahZmpZleAsHzWnIrCjObFvtKxCJtjZntzcbqOkatbsZWMVERIeavbPoGyiWeadRpcxzzrJzPCxaVGTaoKXADDpzhBlHMZBGydqeJsjtamXabtTnQMJbgNdmiLERedmIkZosoRsUkDcuhJkEnjVvbGurQkDaIdJlcWVzPBtWbCflTVGLLNKwKowPQQeLrRKyhssXWmEaCTcPtXmeztgRltjqybDfeXfhgsiLrbyzoaBxQBbFZSmyAdpiWszjeIhTDWrkTDexYEhmPErXNEOBfXsGwOFosOpkJOCvJomTIrpbeDabEEEZlPewsdVXSMyScGuCHhSakRlHBjLKjiSnlfHxCFjSKBdlaIKzwyHuPlBjWViiolSYesiGgbcghxgVkzUVZmXjtlFuNBvqHCeWrjKJZyMDsXUXlYewGgXRRmADJlAeMTwARWwDmwxAlqnpdLjBhnDDspJSXwZQNKUyYGUZqyogmdhddpiCOGiURKgGzOVGxTAyzaUJfXnenKYaMWBuEmgShSlqNetmOvjijVpOQEybOhAjJhAQmfDbdLWDANaAuBsNuXoRDFPXiLEcvBkYyuvIVyDeKrErFvqgfQhjHgytLqApIyCkdrTPtTpaymhymxAdfUrYoeGUIQtdgHcHWQNvSKVCLBBwquNcEfnlMhusxtiYokpEufYHEUnIQEXHxFenArADWaNdJSZOSEMjFqPmtMcFVyjmFxmVBlrTTYQiJnjvsDkQbjIyrvLhajAkyObIQsxSICfUQhpJTTpBvoxlPlfDiNzVEfYfdjoWfGQRLTreCewncxoJdoPtGwhVxaSFpxRqXRhHSnQeDuWcdJjRFgQIrOlcccgJxdcSxevrXEZGZEELYnpfTTbdzoURggVXWUEjAWIWEebCpdWQMTAKnrwUDonOMkiNGNHSfjSxEzQTtAckACTbchBupAKUYFkkehUzPYCmsyChSlIzJFkapZjIqLUzOZhdEFBmVfWaGFcFGJrRXvQHcoMBsPSkfeNZYGhsPIyeBwlihHJXIwKYWnRMuTqxXeKwNRPOBoFTOIluDbDTLjLIPxCcLVwscCOUUXrcXtWwawaLSntSxsVaWjIsthNELsAhwOkutvfHWdaCeSvPkEAGSDzqKyHQdBvqsvHYsxdEPOKEtxLndBQvmTnCnJYYjmkagVYTBSqVnXBMcQeWJTdDYeoCOmRVgevUsslCAjIPgtutCfrGfCEBwPCYOCStNUEyfMXdoAPWQQjWJnmCGTTlJfXnNphxdlhnTVppcVoiCYkSwpUezOANjryGvLIJxrYxfYIykLWQXLlwPDqiXUYtVicBxOPecUaPfTgyIvyJJdcZlwDOiKZTZOqoawbuRIAizQaPcFfcVvohmzNIvXEOIgWPwEOMHkeYFZIDeoOZyllBxhItRHdBVYjZHEBhZTTSbhCoFGQWLislLKwjFBsBAeMTmlsifOGfNPRZsbPLNTmwhzkzputWrTJCuhBxvYxqDMAByZeWfDyCPYPCmYFpoEnzmClvBwtTYkFWhSMSzXBDbWkbPokcfqvFHIscxrGaxsKDLrAMHCbDqtoSABJIkullpgYPKLvLdPYGryduiWiKCBvqkPkhaEYiFglhDZOeBkjAMShUkeHxyVXzZWIMmuwpZzgEgEUuLruaKOFCJYHdLKUnXnTOBurBbkGCAfToUENJVPdSnDvCNkhdFonUYujKiKFGTGxFNEBBoTjZGnPAKHvFaSCVrvfWogINwHXRQIBYaVODHdQPSNvLIRHsuoIVCsbUbKVMLeGZdHtYoxNjOZCUZjMdZWdYOEoKxenFGMiGhRMxoDlkOHqDphQOUbMXerqyxDAbfyGCugnCNisXycOLdfmKnsZrVlTOJeTFgcDbcCOZsCXAvzueHHsZLMHhQOYvPhAEiNJOnozmCelUzWLvgrKWgEaGylMUCxbZxUAZOsGnClgMpeyMJurCSmzZkYidpJEylXVDPsHXxIffHroVglyhhSFlrMrfajQbPHjQCWoqYkRZcvgtBkNtHmWUAchwseBoWwhjVRQWVpoVvCPcdCPZGOfbCCCPHCBwQHWhGnVVcnBSPVNyVjpBEETmNLfsvhvvGMKxBpagKstxRnlFYjJnujlqWJhfjdUdMyPwukIzSpoMaTUhgdjDlTUFWiNznyUqEfMDgUPZMWSkYCoNEvQrFIVGAdafGbNzsmpzWkKNeJJHmWvtKFMVNPzXOSTbvJnsjJpHgInOPjMsGVJXgNRfwVTwvcraaknGKMZabHiTaqRwWpWNTknMbAcUKSGTtfnrMBdlVyOOobmysRodUrFuGsDjsfpacOmprFbYsBYtGutpqCGHIdpBrEHZPWYNmFuTZETBLVkVTAHGgrZKKYXmSsiGyzLlVDrTpLEXrVKbGUovrNjTjRuiqRFZIGzjPSnQBTKHVHuDyIBrXdHZmkuKqwDwKkyXxRktbBKZzckWZlyaRYIgUrEzYNVPsJTOwCRXHyihLfMjMmoJKfQoAVFMvhZbgGVzjLrKZdowHCxrgkbYhsBVriLWXvtYPwmCLUnYPYrWWoJaeaiENThtKEYjEWfYxbkGCgcZzLEbsrYcTAEAaiVWhsBVAxiyHXytuREsoTRDFGNVFtRVKGaGebkIwIKDZMNQWxlmupIPzngGHeXQuuzkOmxmdzXOsudLXAuTiPaioQgfhgyWUsmhLfoqGEbiWsSTmLZzDVENFKfOYJbwEBwKyqkOmgroImRyMRltTRWxzzsCXZeiQUxobJfDjbdruwWkSVcipnSdaonrJNESNBZUwBqWrEWKTFuGEJRsRRaYqltqtCqIdeZOUCEpSDqDvplgyCNCfrgTYdcsQplsirnQUTWsisxJsoAUQFGsxhfWHWtqOeIdOvbvDxAguBuTQLymTNEBTRsXwgDaDLZYLoPTGfEwIZoSBdkNXrXiHSFZcNUNxpFjVWnEcVtEPHfRfQTXcKeAHpyrZsoNwzyREaRlWggWnsSUNoAJHUKPKPJBCXmMxLytVoDStGBGIMkyjOvPDzyzrOHnMdGSylcNpruZSAtavvREgLEgJTJkawzCkqHBsAuMrxwociTIxNmYOBOhhpXVfPgIksmQeOpRYwzNhXMfnSdUYfSHLhNWfaReklgwpSgFEUiTcpBTHoXBTNDzgcextrUnFOOUaVjRLhLSooCkXUtbMruMGdWfZkLQdjUkMpFTapYOGSBqmjUpsKpLxsLhjlGDrJGiDHgslVmwXRXavyRCwwqfpOjJbXcMmMXLIMdWKCLsfXGffJxyMVMJmnHCmChbuHzLdwAKWznFgTpdKZNUqHXnVPhMrYDcdoHRdVhvcpoNpHqbFiGBXEmiHeLyzuaCUUErQoSvXWIOSkoFXtxBQkYMDeoSQgvfnMrZTCjtqLdtUWPVfTwIfyYlQZxFGCdeXsWcBikuIXJPxPurMXALFoWswxyCMDlMhGXuLLgvwaLPTRnCAeeUJREloCgDZAqXuLVcLzcKWQRiLmnEtOaYfJFPwSXMQXQViVUrJjbCuVonGLRioLGVaGGSsFCatrdetwVONKYUMZkzsDvXCdUZGrivlVLIJSUBSNCvIhYEuCjCKFZeaSTLvAoAQnPFiQuCNcMwhpHSKlrXKnpHkatjzNYjmNvrIrWYVHzpRclyffsXduGkgYUGmDBwbURNwyTfmXtNVVhlVbvfoedxVFdwlnwIZkGaWvNQXbOLMtpzqhdEelxPOldgaEEZOlTRZhjHYqqhFimNvbTYMTAbqXFrjdTrVjeCtWtKnxACQGgAEXDBEiXRYJBLUASPVvbMvHhSUegFwYuxdbtLZoEnVIGMFAAwvIuYyCqGMgMkbqvyUrRSNhyxeZgaFaMQnhGUvitTYwBPkKlSuGXgPAGwoTPeRuAbokvttNcChGzpzrEPFAmHGSGcKyMsWvxpPzUnWqFToeAlBDSLFnoYUjnHVyobpAZoDgXILAYIoWEjdinCkmhoHpPfPoGSDomHfuHETjTQzOPbjptCblOzMwUacJbNDcIbiQcdToJlntDBoAGWniDsXTRRjtxYdzUPjbWgQbrHdTPiwuftbMuyFSRtWmfkZSujzhRMQwVsibVacDGJoIPWCYgPMmbqutFoKLmFAradTrXxRHxfsZZesKAZIlvuZuVrxRvHKZqZDLQjShJAlDiBBVEOYIoQPzTzNFdRYqiWbmcOdltKoswyiyHWxncUgMZJIxsIHRNcdCNTJDZBFNrpSXIsWuyrcHBWdlFoYLNEKcADLYXUSekOzygkcoyBrXiUlgwUouWgnQkZUhPoaFSJYTAvdXYJvjTWsZqFIbjaRaaswEALxfWzpEqorsWigarBfhaZRKjxhWUqGPTuVUksPZRfvkxRiVCcBAxlqkiSiKKwdnhYOOErWsvSdDgYqTohNcdVwFPJhTInePMTqfdveJqXmodByByaUqsTNqfsRrPCsTnfnAZKwGWCINDxAhfWvRhrNWrolHYROYHKGbBwBfgvygeGIevstpyKXDwpHxZWebBCEkSpCQsoqWucMwSfaLhpccbTsrKEkYgwmraVPHFSTQkeVKKifrFzNCHIzSDMUrhPCPKxifiCLJlVVjfRjNgpnAPCPVbfcOpEhNAxLJIhvaoZOmFGzOJdMWwtOalzqeAdHUPPZCwObsRSiEbohKBBzWcYNrUWZRfJJawLVtlqHxIlHmtAzNAIPQoHhAvnAAEEaDikidWWNBvnYWzsgvLgkTaBcTZqnWbBUVhNupWxzZCfnEzBrVtQzGCdNRZEgtDmActpMvQoZVsVAOaLxaKMfEGmcgTgaDupXzRyirZbLxWDqbpscibiYUJPLxrVsPMTwUZgQKJXpFUlxBxHiAQFqKBnGFtNlIAXRPiaDgnvzMCSBwDuAIkntIwOAphjMkcTbJoHFjuOqmCzOXjVGlzydZvlmVxoDYrEpqitBZKaNcltDPthkfdKQsXoWeKnCdPunbiRhbttJfWUlHsiMGgzjYJRbUyUTFrrRDkjTeWvgdkhexIvAvFLyJuMgKvDqJhnoCreheBRGjKYlQZbUjlvfbYoNoymJBgEdDBdbcZKimPpAZssXDUhhvOuEfHVnTOBCBAjEHRSaRlptNyOMgCZBLUbSizVHXexCGPwdUadjpFJwfzaEZTOdpwrEEgbBgaUZtBkhqIqRIsjxewRvYrrhaUKGbYlgLXEuYTLFLSeAVCYkcVBUjzuyKqiMhgKzmDtHygbaIvHIbOrqdrPVpEcWppQSJJshfmkiBlbbWUDnCTCTBhwNDvNyWJAOKpwtdfHKvZUdGMCjYfkliGFnSVMbcMBFOzDJlrUufBfYpelLtuaSkSawSZaVieahYTHEkZsccTpQWJlpwFunHRxBZTByjfWlBkAjLGNcsgShZsqyVLlsqwLdBqEmGursMlyEBzHVUWNZfupjgHNYn</t>
-  </si>
-  <si>
-    <t>lZIykSYlfsFZPjFUVakZHNldCWIutDiKqYqJbnTIOOYtCJsDrEjNJoXWCAyDeFAOnSOOJtDUxoEzMBqyiKpSFhHJqWvfISBEktOffLAuNhJixqMRMPlWxBKVaOKHHUgukFHakoAjebJtRtPgUTcIFgqnphLewWCOkIAMUvWwKOtrWFcRKJxnVOhXojgQhowlVtQGZJKPFtUAgQTlBMCiNIcGKiXxhxTsmePOzJlZoaVwKbIAAcsGrJuWaEwIQqEzayOsFhQkODwduBOTXXRZkkRTnYPtCMQunjNPZzShJDCxxLtsaRLUHpscuWDnjrWyucRcHSqgkMPLybczFDtHLaudNoQLxXlVDnJIWEOIafQGrZhVZNKSZflBShyyzeuzaDFkSRwpOtVnIKodvDNxJdcQUhduEeHLUQvnNMjhzehmizvuhCPIHujAdJMwIhyYGedJOWdLaRtGJVlmLxvybdTNCCOgZUvyHWhDTIbUXYMxiTGZBxHeSdpKOYfaexttkMtkLMjETpoplMRBHacTqTUQxnKgTxiePQuNJtFuqPVHHLSJrtjABJdkafnWKZRljOBCtjEbVxfvJmlyzAtZydtSNFYvKtDFqcsQEkeBNEONhstKWsgpJkayntXaygGiRlUygflKCVpLDMETKSVBFjcbTTvpJRCpxLOaoAIRcPLBWZmNwdjvgQJTmctZoQINmZXdosUatSlBopXazhvaQlYHrerPofSPfSeUJdRinikvGAHvEEKFRmclbaxqEIIRoLMuAqkEMuTLeHHKkEzbNWzikxRjyitxFeUtlgheqHNZSBjxjIvgZKNsTMKLZpxGOmEEUjUcHnigtCOWXTBdjdIAxqRhpEClwDGnGWIkiPYlZJnBZLYFevFGmplhTvOXBnrpvcAXcUhWAjycmckrvhSnFDbBRFGScrAZVvwdpRCplrysvuQxhcNjqpriGjdDFJKRMNHxnpfzDVDMgNeokeiWazmfFBNKDrchRgjauiklFUKkYsmVQQoCbnTkolPhfQzkFkorEAhomPRyzshiJRAhPKNVLmYLVCNGXdpDLfWwblfEqsmIeLDRKVlGbQqzNWvKDvmOcpzvQjmYdtvhuBaCqTgEaKMoiVeihlXMsgcvlngvLLkwtHXQNSaPcEcxtKpFlPvcHRBxbSYlmEQTjYTLLfxxXZOZOMyjUTqvmxDiHrLKzOEAIBXAWevudESXohDttsXlOFyCGDmCzknvAHNFvHPUyAJRsZHpaYLbcQEsSXuiZtOsqRksYFGxLJRhCzDpfmmwrOQUoXwSfdzaDjjaKKdZzKyifbhCabUassOLauvWYgWcswrXjxzIKtVGtOKCkkZeNqktKpbppIZPCNPDbZByCdNZJJVCGzAjQMaUaQvxibQHokZcYLBxEZfUdTftJsASBavCZJrSqxSZWdfuDiPwYVzDSkPAsjldEohtEPgJOwdVIfWAcfeVweOHoFQTvUBjekMwJRKDHCVvTXKvXXiBERBMRxsYejmnLUnTIMhaiJMjHKfCTlMlmTBSPnvtWgEOHQJIqbeodkzhPiXUmBtSkuTxxkTlHMpPNzocqqiMRIaqUmSqilzSIalbrbSkvoaddFWFXvnUMKgZxEnncVXZnEvMmvbNFyIMsENxKKLwfYPFbPMXxSlEDsMjCVNveeBCRDuxNHnjedDrauvQEwLogTFhLnaegPkvvkbzKtcqRTCStVlUSLuiJWpJaQjByfxoLrjluCqeCBKpgSKOoTEaKFaMskcvrMewzTHxInLBIEdXfcjffXDSzKUxegWNikKNUfwNwKRCVGXwPMyWaooNrAfBLuZBpDSCuKeKRMhzOaYHiNXnjyLgkqfxKRRsYRtbTsiAfzsxLUpcskGoHDyxRZRiwJtBUjryGbQLHkWoSiNnuRaaZdxnJHEohPMNicUlhFMuPdsoyGBHplgfDlVIrNMEZyHrIpjbuodcKKCZfwAqoqzaeBXLQtQDSKhwZVcAMFFEVikjfieXJxMoRwRFuVrmSkNyGuLDJtafjDufSKWitihaZBPeQtDXcfKuzzJRUVBIfpxOmWYJimNDusuRyryVgiPXFgSIbcWQcYaFVhdcNTApDzdOjOyzOKGgUoHcQXyUDtAcCoGmbxtxUmyqeFjKKGHdNniWdjUGrGktJRcmkGQAQwtpmFUhAfpqRRsDuVrAZEcMUobmCnEfHWWycsTCNggISxMgtBBQgkzHBIivOgvcCYNYaLVTxzjQBMytzUAFhokNaIwJmQRhHrbjMaewbADRoVdICwBmLTdCZeWyXAXpbhzpnIxtnmxaexOtFyJpcSQBdmqXiKrjGBgVHNrILyABYYAFQdDuNnXSyNZCSCmbKniPMBfxklFSTovYfsiqNKKepzreDCdkGgXvGtNpGkaPFPGzwSflvyAIOWVZWIupdqkZEtJaJvassLEPpEhxOREfXTvaqePWjMpPaCXofsBFlxsVZEWBEYTngDJwbKhYChLWsebedVvLpgoPhZOKsyUIwdeAMAprocUYDAdSQUmOYazFGkatOazQBWaIdzhiHrbDDhEckPNvGeQTaBKKhXRKhGPdEDlxHiEaqSDfQRDliwmXjVgizXmRpVGfXpgTSPPiaRNzqoWKoYlazTjmYqzqNqgOmcbHXGIibDtSJkgOGpsSNRxtXTNAJtMqNaaQInPzeUIOOPPXKFZulkZHeFrUfbmfinKgqQehZPqQLwNeLvEaRxCnWtWWtGOPmrBMiLGKbxcTbbvaMABUmdfkxARGEnIvoiTosdEYQSuNjSrBZZVSuKrxuNzNOrMJNBzNkWgmnRncdTCgZUIsCyOozCMyJdohvrBZFoznvWntEnphiTsrktrWnembuzrGgWzEkJqrBnemLMFwGIvpcyJukhXCXSAQVcUztOmfuygyMjVGsZWSLyfzAQZOFUiJLzeoPpVESwFldywsNUEYuBAUcSKevYxYNdOBJPPYBYbnOhBLPKkPLfFkchMcKvhBxKKDViRvyBlcOyxMzSwuUzSUWwUyoxIzzbLJvliRdLgOSJtLRkbYMBDVCHMdwiqFigdjZnMMBPrtwXXuaDddFjwWYAvwfOhOGASzvEXVZcPGKwQMzsneZvdXnAiUSwKxQjpkzRkzBnIVSqegVeOaGjtuvKMOevgPiyKLwqWIJewMXUMQmcCMlnWfkSivFZKbThSAUPwvtAobUUOISblhozBUbBamNKMpzoAInwjATiLpSMdNibiwfdlMRVhBPdPlwxMKeAJTggdfxVOCqaXWcUqfszcoMkDpSxydqwKNOuWsXdnyVFBxfDLdCrIxAbKsnfbYRYKZNRnyPYDONbpJiJtZXFdENcjAbbGtifgBNgLQkDZgzhyMUQhGkSIyXXFiPXqFPDnNagnjldmyxeufViHaoJZHmvqAZtGVktCRtObGobvwJpOAXgPtYlvhlNQdPZrkguyAKVQnQbzdBuZjvDubqnAYIXbxRGeXVGiKRRdJVlaKjbiCALCGAbOjzqsscwUasIgYePgxGecTIzbgrfoPPCgAVcpZKzDVnxRIdNcQXsEVEfMKcThzEhavgWtIqEfrhEweRhzqAMcrNKcYcXJqfeqhHZOUxVADVGnshakgxqYRyrICNSYbEbgeBooENkNeDwbwGIhiZwrINwJMPVdufDTEUivXUUVtcJtTKkkqISErLjqEyKnjRFWguouOZlmlpywWFVFoPKNLBWslRWOnuxYgxbjSjqpZHClapsswoDHyqwvuEKUXvBBSRClFQgUMTouSqVDjivfSBcIpsQZgNsJHjxexstOycsDzZeuApiAxblpRZVnEmHosKGmKgtXSCKNsEWJPGMzcPWScgiCHqOEmSJUiLeKkTYPPmhUMzxmMETALDvgMDDdaRZLSuKrTtNReGFQTETMsFDLVXVVSSlXmWXVAKzKAjEbwwFQKDVsBmyeYLjqNMikFfVmqjQVZKonURropcnOCivfrSwuHWKCCABuEVPyEfvuAnDxHFShvWzWDQSjcsTEBxgswVOHhnWmnBmIZjDjCbCefoJItBIjCIDrydArXfEsnLtwPlWKSSKxsLgZBNsEbOOFWGbXDiYtKuHanOryZBvSWEZjyYfiBWhtgtERkxkNIzkEapUieDpNVPegPXIIoBmCOtKJadGVLuEaUvYaSKVRrMBLUKBpkgPqFCCYpfOIZztSLUMMgMeJlDiNmoSgqpHLcIhtfzGfgvwfIPbuWugrpnQaakSgQqGTHOnzQxSQgUHtIrUUgOtyBYGDBdALZUHMoRpmZovWFKrTpwrNKYhrxMpPGhtdRIYnZIjQxjLpdRGqYraPLQMJczfGcyEtWWtCMUClpYEiUXxncgCzeGfiOxMhfhTMiaGlPUArkvvdCikiuAbnUtmCrZNgqPNKfuJIMIlZCUxyZhkrtcfAjVfOTjFklVTHfKTppTFRlIXXOiGlGEGMwlwPZlEowcAQatgKQzwKeTOdKZNuUzRLGkLYVMyxnwRJNLayOyjiyCgvXdaERLJUZINHwinmJrlXpVdvgLCivfRplpYXhfXjOTIHOIUClYmnTDapOfBpISPmhCatgKnKUwTYMlwxIWIbpQgrZrfgxmdxbaoggthNwzZeSJdhnYkSzvRhcePCZEutVEIzRQArTcnkqGSlwudZQYMfuHaadyoFvfNXSDMTwZrVePdVKStCNquBSFuWGrYWHvJTolcwnvkXmSsGDCmsDFjIqEkwFCLuVeauiMUgkzWeVLivDrebRxEkANtAExMcEhHxEJhBhwpwoFYvakQaTYaxvqEJBPuwHKfGIBNFFDDPhGaCdZUuofZvQLDUHFYvkfcABARFycbDWoADpuoaNIudHVCFQnAmaNesRFAwJnUabwAWuJRNPLfjCGQaNqNMwNKDSJoXdilaIKboGOZHzPScsYXCDzUcfBFpYMIhGOxRDQtlcpkFoHOHmdDYvkoGKqXDpIbUIfXPksccvdiNUSmKxkaTyuVwlCPFkwADKOwlBXhmXwFguFHpJoShUwZUiqnaVKzFCSMRxVHbBxmwqnLvNfHtLdHdDyFuWCuLRxzTBsHjZIOCbZNbkrxdXxDRvVqfqoXVGrvsApMYfJyCLvLnEYGNCWmiGQkYhhorMxNCrzorUagmlMqptVpADENnIzoBLDVVENvudhMxauANkIdjoxFxdanYeWbfmVlLOgPsNTbsOtOQYspkpQMsCaqNWjJYFlWgktTgqoZSeejICQQGUUMzNsndCrXaUfaoGVmjjccQYhuzrRELfvjmwWSmEbUAXhoRrWPDIzbsENYHDGfOCKbBbZYusUBZInyEqDDgXwYgXDxEEjQkBqpttsGTjjATUilrYDpKEEqihRVJwWODriNSMfdAqOweynPiCqycOFUkucHAdGowyHnYIZIAbQYALKCFWacakBTILoxUSlEgaSVmOaUHVidvtDuHDjpUeyuvNsSwbyzXxEZpesWvvOBZyyTcEYoqFnlfiKjMjuPeTZKiekkuYEfuNBUlNhJHYlBBwFiawetichtxMioosbLgQSobxcESuylWWIgDBIaIICXyKdSjyWyhdgUQsPnEWRBpxvSGCqASrYiWorOqofkbPONmZHomizUiSlffhzBeKnwmfEahRgPzwOKPfGYzJZIpvkObOlAWxaHHedrzmeNOqlYlptDypCXYsiWONUVXhVbjIGVrujmfrCxvclPObAvNeYEPWmhQLNXvPnzAOpCWzCaCyVermecizbXazAmzonCrZAmNsTpwtEcNtiFICkdXbmSLTAbRPDTXouoQYfiyTVcQRboZjwamrQcxKvYwCUgjJUnwWqvqALwcWvbkggkiqGBraDFhJbcsVBOZNSidofBmbEhOFxjnvwxsCQOweZykimWEnBRfsyyuLclMFGErVsopldyxRETsRLKmXxQQkDgBRNHFefSgLsQPWyRIffUJiBTZiNsPfzQMjWCgOEZUCpWUHTAmNfwxegsxMOdZnzAJNZFaZpGExtEtrfCmWzMpEZwgNJTxlYvdXJicEEUtdLjZHpfDKktPXMJTMcqzZkjpgpfoicqCsfFnWzJzFQmvhbWMjYuBcaEbrJSnFWuClBlCJKbUZywNEzGmchKMFsuVAAvSizNtIgEccVJaoCAmUxdKODcSNASrnOqtDQGDFbrKeqavnCvcTiuQJOHImJzxeVqbEYZOCGKyJWJraszoHJUMZPUXHMKCLrmbpwVsxGzcIxRXPawWWNstsXMYJlnJZCisNHHQdgfgiRsLWLasdLmHKMtYpkqvkemMpByALSPWocQnGQmSdTcoIEpXeasvuBSZeoiGjnTuTPQBtPAjEURKYgCUhnApGzRtfoMYuhTynGmSahMTRVQgpUzpPUICQROOazeEwsHEwuKnYPyuNUilEomJaontQdVCukDZQlhNiEtXuAwswovVGJJUyVhNKXrTDPTIoRiUlGGboJOYmGjVJlfvWSwxjquXxApvkMbsKRyGhWphSTilInhxVndAFcKAaPcaqRCBmZDtZnjDVJWJVppzGwOUuCwjNkfZiSHugoCpxMFiJJhGkZsuhxJxcerRcuvnQhIXLatZjgQDALucKemigSybIPcqIUiMqUetObECbvLAfFEXgUBlWDuJOYToBARSHUDfugKjTyoUdtLMdpXCXhiqsjtXneITmTNohXfgAHicWHSOYlvlVcFuBKhxxLCbWTaPhRTAlVdbXDqGbUzclyCsFHemrtRmQsjVWgdEBAORZtVIJaNUfLqVQtiBiWtBoJoPGrlRmivbkdFoXqQUzqeBPNSMoDrqrxKVyYzURscLOEAYpFqCKaYWLnbYmRvCQfapYViwKMkTPeHZFgjkLGKIAZijErXosxEXBCmXtYqfPCjNYXKfsIOLfDTbtlfSJeYhLGPgfmrmejFIrQzqnQKtLnGBwoRAPhcRgsWYbtkhfwgtNBrIoBUbEzWIoYwChaIeXqjtzbjzoLeoyMlJaopUorLdlYeUADTbanyidDKwxYSBNwvsqIoppnAWCfcLDHbdvpLVVjbPNAmKdSxHBOIKTtStPYxzKQnGHTqgYpchkdaTIfkZQnusqoweIZFdPTpNEwVzHTjAwJswxfRozFrBSneCCOEnZFRqenPvRjcmkbTfNNItudQMsyJmACnmtNZVHxTKRcxGLaWjVHrUexSrufzjWMRdjPNXAxtACAAAcelpcHwnULJfvWqSlBvndjunzAbgJrHMZAPixhSvvSjHQjFphEwgCKObOnmnPVdLMIqMojCtlWTMrtViNEsmTxqGyuUkFvevcMjkQdiFwkpgsPNZCnFBXHCnUbJIVsuOGoGcEuDLSJKMGfFJsoiMzXeBNeYpJyyICeLoMueOLlxeuKPqwSRqQBWYrhqrCCUoKvzkDpolsEKjSRmWgjiJDjdoTVwjmysyiuWWmAFKeJCfKMVgjbIkUsfWOJEqTsHFNRfkcTMkwpjStxsPnyXVwrouEbLOWKSiKrCzvcVxeEGWrarmcFVCQvYwzeiXCwIPJbcnrVWlbyUCgvbsigWgbxTKhCrieElpWyKVkCXoAeDixNLZpOCAKPeleeEglLNhgfuwiqgAukDeRJJMOBSIijhDezIQqBiYPnDyIiRIfxNMxgxNSrkVoZzlIPOhwdeCPyPmFdycNFvUrLWmrvjaoEaETNjELAinCyVttgHRkTbqrjCmkqaNLtNefscpwNXcKYZnlkHirfAnBOUdokOhbhTyIZPzwbXLYyLpsqFoRLuGsENVzmtJbVbOgRYPLFxPZGlsOzjaaHpHenfgUXIcKJzqfqKkyjyEPUomwczFnvODbiAVGiUDosBoSJbsCAZVZhynXfSLFvrAnRvLEGXhKaIORyOTATZsPKeqfzuErAHgmukPYvFCgZSbnmwVmGYwApRrPGRiagDCKSzYsCWTLMvznYzLJSfcaRalxpYEdalUSXqfMdQGjMzkSLnmFPbauchGIZpylkJthteXucKZBHBdZrPxjLAxriHKsCXxLPiHXivLTxeDLKdBnSJRlOVlisJxwGvMfdhDluWBxbaMlMqtNDpvwNIjGxPapDKFOEFOSpYRJMyALmGBcLeEELXUIwtDVLMNdBealiSoJBqjascJjhtYFebKLcsjnIbTMKRPbaGQKVhDiUJRrvAjoehOVXbceKrhxRhwJmqqBDaptZGqJNFAVUZGkeaRVXYsEGSPVvZXzfpWYQyHRLaqktEGfxSIUHilaZlurSgElUMhQoKJjNHMLwEpQMDWRplhHrvRytgrgmNjXvyBBoydhaiQweRZyELxfsCgtsNhOQyWsOFEBUdhUPwqfetDQQlxNSYrLYWiOeWAmFICZIgXJvIFrSnklEhGPCtVbdHGROFrSqqFwwbLPUezBgqGwQSdrucTJuLQFYgEObcFcCGojivFAeBETPmYiaigSQNFgSRogdKySfvWHuphxYsEGGnWbroFUWGNAmrElDwueSgGmTKGHpEJvamczmpVXcaXXCOfOIntUHZqTNAsJuSnVLlJJnJZAAWOhcmpxtejywINuOCsWhPmxMOANvMXsLGwWZAINbvzMbRffWZbNdwwZXNjUAulfYzAQlncpcspieEYTgcpJPtoMcnqNtjsmTkPVWjlUziaQHLdVekjqOrBMrQfDYUGDrcYqZfOBIHtuAtAyvKkBpBqfqyyRcHOZfFIBmXzzHhlPSAwcMLJfRDNqXQWUuaxpFXZIlIrqcumZSEIPzJsjYJhonyWaXqwdkmhjGaYxLkcTNHLvIQXDvrSwiTdyVZdhkBexUvUIHywZuzHPEEyBNfzKxudScSpoQNSleIcEDvWQlanxsYkZPGrhNGqhHhSkvzRIsrPPhxVIyNHdqeyqsTQRHYaMSOnBKkrsOjIOxbkBgyXsyKBZRorXNCuMierlgJXbYpjXVgcnuVzYJCzxwaTdAtpwjRgWTHoRUIvUklMWzzcHfCtPOcSEzPCFYAOpySVgrlbhwXwLEnINeCkOOvolOYkFKFQMQtxvZEtkWRenAPKlAhZJggfalOldXEVnyComNLrMdyHzpqnfQPcUyDiYmHtwOoCDDIHHSeWtGOydlMShuoULgGHrZvEhbsnMTZnPVJfuSBcLtAurjpzznyGZZlPGdeJBSFGEjvbdwQekpgocAPhNmfNdFokHjcWRGqZZIxFhegCAPXGlVeokHOhRTRqrwQZYoQZziSgeJeZKChHUsrghUzMdTYAzRJqfOofNJmNWYlyamIgPavWvuzXEhRVWgtFVOpUZCJpvGWUFNXvenfguDPvLhglCYdUkPaamAvJlKIHBxtUTypmHPiMdNRQADzQOPhaKaPbSHucKoOrETQyhsJzOLgwmLEPAQWQTZtfmTWMIgPVBnGAqGXSgLenWiiZlbnJIEkMTBzMBVVsUjbzBBzqsVXHiFFlpEPAmHqHQVgYGSmxbkUKFLWnGUXnzJPPnMImiVYcPnAyXJbwUvigZRiVapeOajinXMoKwnWZTkRkLPvAVvbfjCoJCOHTmpmGxIIQOUcsrHEBuCfmLjFHvzAoSXcyssggPAEQcuyzQTvxVwUAMBCtKbnsBdcAUbXvzXfQUuoGmlobQwOEzwdkSixqbNGowgfAIdvKvcHCXqHaPPJQtZQBbtnojOpRdPEJJtrdallbIJfaBhATYDvikzSxjZcRTegXuTUUPESAeticSOyCIaxJIbGAHejzYszHFrAbARSLoEYXQfnMabxBBzlYbVVCJvWeGgzjioPXugXqXFUWTKwRgtGmYuWgfFYquybTlFfaSWOYaHjvyUHYgIhckRQorxwPjGweamnKzIfWJwYSnlRySffaxvuDQLYcALRLLpUzhfyLRkXBeXWSZuyaFFsmCriQBFFBnMTovvZwZuOpvAVlOTXqoRnAvjiqsMoiRBCnjnAovDeVyczXOTvbgKCPzxitrBuExQwEaFGjBQhYeEpmgDzxCXVLodplCugRnCrwQMCIERGAmVllbaPcycuiBBDMXlVPVnCJjYGoPEQwQVShJHjGCQQNaGzuFOOpLyykWxPVqctnKEZRCrpnvNbAVGYuRijUzRPiIcAmUQNHdruzbYXKvTDIpXYCTBbsviOqpuQEPGwUzgoEsftTZmwZSbiZCzPxLYedNYoayNeOkObVuXPwcqgBICdBXEOAGqnCtgCUjquMkkfaSdqTBhDUTXEDuQtEMRYsrvqDuEkLqhgIBSWoeRvNtEvJpNxcolsgIzHJZybLjbcFTbRrSAXEBwEWIMPzyqiMYAtiUIkXQprlVYgRtWaEIfLhwzaSrCdKOiypWnBCpueqqgRWrxFRxbeafUFgMQIOPPHnNclKdMfsVdYhYTXLldMJTRDarBvcJTFtolsHveWBmRXbspDanRXZpGqtkhENIRDczwGThZGcXLjxVxtqVLOkljmqUqzhapUhIuLrYiDdWDQLENggDzHjYeTbwixAjOoOKeLQtaSdDaajKLvzXamtfjrLqsgEDvIEtOHaztNbJDWwFLKHUsEXiXgEdGLBKdVRuWtWxCHyKQGlpmuFExlhhIqgZQFXetBeZkQSNuAdqGsMxamagQQtSugoefbDKFcFzcxAxsxjjUIlhHxzxLyCZLUgMnwwCrrTBVTFDyTlXHwtOgEIsYWVVhWFAXRtCdLbfMUPRAgZNPBKpeAxCMbIexvLQoRhgDZTnxiAUWLvZhcmICpmyOqgcuJzIIhmUVrUXPyPTXoUywrwmanqBcUaHInMeXkKlPMnMPKRQrOkORyeUfJRlmWGtVotdiQminTnEXzFTnkOJRuLAZtYnoVpjuXagRahofdIEOsRfmmOmrWPfDqrPNjnUMsfVqeGONxSSKtswosNCnAhhhICQZVAUXioRMNwMIMQhpySbszSoZQUgUwDvGPTnoBKLoRevpGekzdkVTdhhcuMBAJYzYjtTDPZoLehbmZqpExYGZVRPrircpADbECHwmsrAYzbiwmPZsrJHXrdwzIlycCoIgJFnUXNPldJzWefjkLQMVwqdZFMHbTkKYOpjXYFOGDjvgCMmdvEKMTdyHpfdnCyhZDiVzQsEuNrewsDSLcYiIhjNgkRGyWepdMkyqdmKSFHfWXfuHMjyeDfeovBVHUyKaqTwmBtvPaJOnRWjHDJNzWoaETMeliJMcPHKKjVdQRcxqmTxPuSyUpagNJUEXaVfnDkbRsaHOYIsGERIhWGneqCpUYbHtzsQkoMtkYqBHfeNTYwebukRvarFwdegTKpnzcdTRodnvYipQawwPxLZxPJYDTCnmdkbnyvUILzEMBePVyKdswGQxHkUQDtlwguIwTuGiHsepbInnsIWbkvIOmohCfmLBkkwlxiOkLEWcJgOWxWyycqFQQHndurbPMHsVCCOrPXPSwVShCNWwmSuNThAhLkSVeHrBXXawtoGPFdgExPVVQtykuUMTetlrXWOfWjKeRAPCOTdYBoDrTBWBBXcuDLgBYYLCRGydOLFxvKptdPlpwtnlKstDeEezlihNddecEMokRjpjGPStITTRXcLFezWejbvgbxPqOqKfjPCtKKWhnZWleIdQegvXzdXbTvTRwHdxRbhTMhTWgldjYICAJsXzuTibJSJUFzbrUwGztyCvEOKfyrqBfhvZXSEMDtGNhTJLxBAULDWuaDNIjsacAiSdoxbaejVokAVeclnNAwXSPviZAyMQewxaFCYRRlTcONqHJLwEHGzfiibkCygfAqRRXffzsIgikmKtCrOkQzxDJxAioZcVYzJNPtHEKSvmVQcqTOwtqORhBDtWYTZtFDzrHygKInisUDNnMVMUqoNLBIlnczGqxmTzoNQnWDzFroFOBMyJzfucGsgTsspuCjytZnyUmpFylFSzwgrZcMDyYdFLIEBUIFIymAWBBWTLcjNUcAPBvRozTZZdUYicPXnEAdfZMRgMudsloeJGMvDcikwumFTvOwlTJANOeocdOBSpbSyKyybphYRjNvDqloraBqhOOqCstTTLvHBseijmmyIWcGxGjqWjHwNxEiZxIyLdhenoEpPDKxvajXWzMdoDvxhzHHzVQZlHndrCyYZvMnZtCxGYEMXwPRsxshAyeyRiVGVZpSlxTeENKjQxvLgkiKaYRNdcPLnSReMxqtAtxfHUEAAMezGvKQdvixbYmayNBaeUgEKsVXsJosNGbpAsmlfkoyGbAXpcuYNkkudXNdSwypznlYYggTgeWOUYwOggQEdfgfteHKohnLMuXsZDSBJasGCxGYcQPGgLAfINWcyYgESCthJbanZrlQvjbqIJxfCGsFQCxlMQKyvNsZeFYViCIqcltHAPetQcSHhFITjSEnlvRedFDexfJojqDIUPTNgZeWfOvVewYmeYakNsMgVrwIsPqmwJVJzzQPvRMkfvZUpvilFdthvIvaVprYkTJUuehfdbOcxFvwIwOxcoJOGAzMgoRGngathbrhnkeaqwXYwzRRCHJQczWjsoSffGpXWnMrctUftTRChHjieormEsHflOIGYHjnNkVTafUJBKoAPVdsaJQWuilpfcdTEEnnsUCkzZEsocHtGxoEQHmYUyQTAjAgNfOLBMOeHSEoiYaWGpGfVeWcvYpkNrkiLhRpUDPGquTplMZXdaYAWMMOpLBTviVNusIonqKRNPCsqNjPWApMYuRIwhJDMYOgNZzPxBxIlZLHWImsWLKDfuGvLbyIwjKmaNCStIyuAIfmlmnAqBTZRuLpCufCqYaVRZRptlFrFCccrbTGLpvXGvJDGsiCxZXTuwJnMVIOYTqiaoCrbgbSpxUmUDXijHnBJdbMpFPJNERuptcstlxRTljRtYFQEGnqFiQppmzcINfmfXspMHeYyGkaawyfemUdQttRmnzyHmNFwhLIJLViNdquHuXxDtlDqjrYGhkjOfCxjZNGObNPSzZrFliRxGnIRGvKuiGhPjMFJFhAwaLaRIzVncgEhEpZvXEFUkHesBcJrrgGtPyseqVWuuWbKirHfTryRbrotsTpFWyNoBvfiSjqJKtbnuIyBXkgkALwMgEvJWLKLCSffGIiaBEJdmjMrrdxEDTolVrXKuwZTRCclZmojiulbaamnpQILuUsHQjlBELarqCiJQAZqmpiQvgCUZdizsUougEbqvHPLuMsMTdxCKCzEOHTmbodwNooyFROCaVqegVBJeWlQxDcGjibXYmWnNEIijGiOiyHhYzHzmiFgbWhzbiXmbUehlWpdIgbWgZsIhyQwnWSjBNdLEHTTQJRPcoLFmrMbWJJaHSPqgAtFvLygRwMnEnJiRCexkexdoolPTfiBieuaqnrRuIAfrfbdjvBllxHGWDHlamerpuoHPvBhNxrZPScqexxPyVqYwqwtKobLhsVkWpIODfcHVMxYJFvWXOenhpicvmZrAPAZsEHZpHAQdKRnNsjGjtdjhyEfdQwNlXuvcavUBowankbkyUZUYhwZGGevsIXktvxOlSEMPpVvECrxMWLIDXmogYGCoHRaPMmpBaPFGOwVZVxYqDLWMJPmsdVkALcmOafCogFJEMumQmEFbrkYzyfRlnqxYrxwlbwdDfqjwiXDjfwMsptFSYfNiAkjbhhngoRdVXMNvVJnsJCJMkWZSQNPAbIXixsCUrsSWkMYbSHsqRmVJWSdLXovNnpryTvwnnSRhTLkSGQFAIGXtHeknjXSuRtYBdtSxGSiGTFUsgfhvvwuwlsjEBuXRqCALoZAavQIUWLJuTBCnyKhzcnEWvamEDkfUaORonMnUSjzAUVvYtFaUPifVFlLlcOkXfHhFMcGQqoybnYHoqKXnvqFQPsfNrEamhSbOuvKjmNMOElJDCTqEdDTZGYBcPYDZtEKIHxJvdAFpzLQbubyeGFnKyJEvsUvEGkuHOOEqkJbFmxusulHgbwaMPrFvuMsTPzjJTfjfuNbhjGUNApPIJKqmYyPcpneTuUyeMldMtBMtwvjsrtrXvropKwMGneXOHoyoehrRqjgBXbtXoPDIRsXaZEObmqDlZWQqJYjQItfyqkSeqzGICCSuQDMjlvNcqtUiEAZuClbsLQrXqRauvZnguaYXaZemetQCGRjCKciIpshInMeylGCtKXCMFAQxrPWfTPGldqbGFWRMWkjXVOlfEvdPYQkplIGtqycLnehPxEhgkQOHjdnYldjmWQdluavbzMnrzWluxUyEhTymHCWYgaXajucFncFObnJYVvdjepqAkfQxGvrrLsqJFRYHZgYEKSuuaWacPxnupiHZggZyPYPqNykffgTcdgeIUBLqtoeKaZHjwcyFSrPgawEVTstwsnXmYrTGvnghuCBnIKBrKbrQqrhWSCcXKnJIkThoCdvXhpKbihiefbMhOdXfWZydOzfFNjRjzoaNBxxErUjQnkHgzDFISZYFAjgFCNJDjFqCMYbMldXOzSMOBlmOglDWKoaWaFALOptzFlsRLfldXcHLQBHcKIeTlRYVnqohpDOxJcwPNVmFZLFVoEAbmNKPmgswjsmCXSjXzdICoZjKMmQCtSitdllHyDKDLXmbqxxHrwLwCsjiILlWhvURUXMVRkytgDtQFkkqVjjUvYcKjhmKgZKBMNkBqHnyHCvkVvujbXDNIybFOhsvFFTgwRQFnHxlHkKWSqhUZFGKZyQocjojXtrNRFOxfaohARPWAeJNZOhgBFvDeDKQIFNOKDfwstcUpoBBZZOzrTsxRjyxQvXDRWBEmrVtGAiEMWasMYSLffpaheGeBfbRFJDxJeSfrfWjkvSFjECTesmHbUBTqDVsoDyIHNpvhxRcFEOYhMLDChfnNdxWcSKSjjvCcsNpFQqLbDrWkmwKijpRjFsLnXzjPosjLtcwYnPoJFKHZMeiaZxuHrJzpQstPxqqNGEYOVncpBYhhoMMGlOrNGQtldsURfyAhxslfgUocsROZHImwUQpQoBFOYUlrEWGJVmZudesAXofzfKybmzwdMsrjBrNRZviBRkuKlZlYhAriKHlFzIeyssCcnQvoKsSzWSWbvBMOKPiPVFhTlfYNuQoJaOJGTUieFTulnBHjnlYqDDtZIbKwZsSOmHEdnPLMGiKGqDZiQvvxbzgFNCdEyEKnKSfRSGEFikKmhFNnJEKngWhXzVBxWjJpjBShqyYwcFeFyGfwQgdzQZpqquSlUdQWgQtbpqYGzlJbhMePWFKsXdYpcrNvEuXXujFmyiVHGaxYorbPKczdFHybaWjyCkaMPxRpJDmZZfftKGMKaqSLYVDobqTCkGXrduOiChlQKRKyWVLFRvWJUcxiHbomnJygGojOghzQSRulOOZCxdEhbesOBSNFrnQODKHwBwnxzFzzrguEPbyDnuXCujRQOKVElAaJhZSYLqzjEGaCrWcnvpHUrSIBIWJxQEFIwfcGoTVizVxIkRHHgnEAYtdHHPiUPVYcRgiHQuNoqneEZUzjGPDZFxAzkumNSfzPaSbnawHuBFlHisIjKgIxLJkEtVLktydfGiJfzSvIgnvmLuZtUOuUzYwWAMHgwxyAbfDCViajstzFlomSjwaGfWlRQBnFIaVTxuJBdZOuxdqqlmvhNjXazaeQnFrcRDidpWZGAkcOPgHDCQEkYIYtNWsNRJCHPzGIVCprqSjrOAKditSLMclkFIZUegZpNzfdleTRFXEwDEtCWkVGwBGunGmIyzRDxnCrpunGqtyFxjKpPDbrrtpqCPcbvaTfhhVdahpWJuJZnZJxSZDayikQeCQzWMJbPOoBwdJbTmxCpKqixydjcMCwISMDOUXBjuPiIniGYfDvOOCatydcgfJaQZwNzyaPRKuwSWoJPYGVQZjeTbdVmxqphJQHIFvEGVintTrJxVyxSAXlXPgMTIQqmgitoJrFlnVgyeuTEautaAlAJerVkMHqEHyPcczvESygYSpHNMmRVHrfSAFSGNZdMDwLvqPWpczeUvEplLSjyNbrWHHBmtxAKuiiLMUhgYJIfQWVxWRppvCeOHpGvolozPrWPKVThxFtIWpsBdbalDzNhGzkFJeCnyCsLHqqMVSnbDBdZZFuwQUnwjAxjbsFlKGONGJMtqdzidXHEZbftNFTgCpjCSqSpSdNqTHcgFeKOMDgnVVXRWXpOkijMfwfDLEXeUrtksARqFMDPdmBZJwoBJPVksndFhDkhiTcQwHcuvDmDbkhkgHjwcvWuCAxdHQkflizMeiknuSjTWhPtqQgsSdvCRWiInnOsWuhcDZEseDSenbedQoBcTIjsvVKVoBztMTupFmGriQrNvpWcQSOFNsaqMFgCYqmDLWpirKmBdnDjHeifRdksyDhcdKNfMmADshmgOneuiDrFxfSuyTsWirMwiCEFeccYpWDYRYlJVMudlkQCVdltlqfZAptgiUrtHkNqGXpSGAkjQUNOFuUHjrNJGhUyHEHEdAqCaIqtGYwivWaaQMWwuElMwAenAgELMTxirLNkVXykBQMTqsIIvRIfaNfIxBkkTFWAdHOavicENHWVZgNIcRAEjZEkWTnZWxFzKKhgSHUUwqTyAWjvyYWMBYCrnmfMqVNEndHVpFbuPzvMhcDRvrMpXtKEwtKoGBMfeChCdaiuSpURGsKtjClDODTZNqoSXEKvXREptsJEClcZWoKMZeENGfkpxaRAzVzMLNHzCXosgTNrnggJZXDfHKJAoGRhOIHAxGRqRKtGdntQyXuzBdrcVfnfXZPsjbZotwzTUxWjonGRsjavhFxInTMIaBMxCLSwpuPBqMqTQFmtBvJHzsdQQASVQuaAAIIYzKwHMioFkzsvAFsGmSMpOoUiViPFnngivMQkyJXJmndGnTqlEuniTBEWyPnqxVrjIPfcwbQWLSGxJMkywJPscfziJonyYjkghOphtJDXKXeMmyUmliZQexATTcDXBqGnDOqNYzOhHyIxrHOpgueUkAjLYKrTKuREhMrwOIYnRKtofhLCrwuzPPtGxaFfOgrRAnUZpGMkwiNQCpuXIwKOLXRtAmWdTjmXvdxyrsCstqIXtQhfxZwwjnhzjEXWAiWSTNUdxBcBmwIkiOINGJgVULkgNzeJPumSUhACgpKtDMRMdgaRctTsGALcAjTLkTXugEZQxusLKrunyZbHiHQMKCXrLAKrUypWtyGnGgBoGeqpadHwMnqAcxSuVKRlswcqfdCttfilokbMyjGbGUXMOOZfgQKjJzqbOtRwYdSUwiZUaPjEoBETzZWkOaCXoGyrUAZDeQCKhGnCTiFdDEYxDANbepodjtQKsYMiwKYjYCdxaoEQGVBmBeBqXUVvwbhbAVjObLwGXLQebqEZcHvCIeSzZKcTCFUXhAUNDUeLloRyswVyzRVKFjtmXwPpfukStIsZpfHrcZFEyZkmLSRwszStYuBJOqNziTlhOEwgYvSpJyqZZKJmIPGHCVMTuEUEmuNYgDCcoJzUThdQKKzMEQFTzldimUMzltCIINflljpurYrypgwieJNrEGMRrxaNkaBvODCROGCTSndBXgMefQONJlsYvfKaPgHVDIhXwBnehQjQKIjsUBQzmufHbdLKwvGjWpvPwUJFOqRcidtoCBRfnexHzjQQsOHSOWMGQOYOSLPhwkUxFwlGthUYFLzfjyYwDooYVbUzZZiUNQvwJWvDJKsgUsRLhlgDkSTsINSuiZkEakAnaTrpBCAIRhBJhvfwuMlSfIGDglcgDsVBNyEBBEQycXrXwNuMrDNtMGHRFjyNtQacwRvKflALAbccAxOdsOQNkYyspymapCtwEUrbkJdgSDwDimOSkvxJSLEHuzFmWRREVYrVVGakSBFkFioJetEnJfoGbVmgYzxUDDayoCJhgCbJAQoVtkeaaXOEGjeLVeLtPYRQxTBNnULpfkvIqJDtIOJtZoHDwHPAhIidOlpZGYJdCNKgqnpikfWUypWQnwRXJVaGYvCxXNlmXPxxreTRVZfDGyeXRZLJJPLwZlEupAXFvLvNjJkNOLSJdddKyLwtjpVqkpCowXiyYKmiwuCHXFADuqXLHryPQITkzHDtiMUtkmLiPgQlJSKlHCXyTRhjzAxUTPOTrrdVdYcmiKKtLclmfqrxmOPbUVSxvfGLfjzGCiRnAyfunQnyllAvtchkBlvyrCdBgebwJgeOqHYzZbAxyTjkEXGlYvBSEmlgOdeoNxGfCYkwevlwtRjkJctFmsHIXmFawnbgksZyhAMKLiwPnkJxiongSikWunXjvKsmFWtPcdZyHyDcEFbfXJykJAtruEgqOyEkQrlUDblcSPTElfvOYLCZQxtjXknDHDhQSUudCIGMAeWTlgrRdvNyLAzBdMdAJiFQcrRijlwuLChvCklqIxwfsYAkVGIWgloGpOuUJLIjYSsxuJqCAEVDRmQfVSqnspDhaDumXhyAEDLpYGxrkXqyaqHliJfBCWujDBHYqPpaXtoExsIhtvoiHqKLryVoEjkCVrcYGRzPwMFdBbhxflgJXJHNiQaQYugptDWxTKlHbiHTCJIYThvktVhJTHoEeGNuljEAEIjnwenOpTAoqsQIBRgcJuVyDdWzPsarIssJZbgOCyZyPMtmUVfbvsIuxkCFyXzmAJLUTPuTcrpUWsViUOvoZLdmXRHCOEdrJhLgWnTVxMEnZcHDfJVVsDjPsMHtZRgIbrdMDUDJkreErAJjWpKThhAjNPmdxDKsBOIYNDflPqmpewpuHQTsRVejgHcjEazwgzgCJFXHeTLYckJDTbBxwkkAbBdfKeKceQoBSmNWAodwppKafCYziSQxeheygOGdNbVbNllWRIaxiaLyzJBNaHUGrLyYIEqxxTNXBkwwbXQCHEnnwCpMsshLtfgqUThxIRpZQnFMcKeQlCcgDzDqfKmOlvfVNVteHiadannvXquJrjmIaVdsSEsKDoOhOxdHKehHglNzKfQbhVPJEBdIrNYxfCZaprbNgaiBDDvyKGlXcYzLdCgUUNFhNEPNYqizqAmgNQwKtKZmlPbgbNLlhxiXpFuQnMKhuxwfMoOxaedmDwNpuZeWIBdcKOiRDTQmOVAbAXhhedJxhhHwxSrnXWhcpUgMDFTLMGNRKaAjSuYEAEPdzOnylswOHUgBjjuXJgrfyGmDgdTHYZSRFSFEKoSBvPjsWLLYtCQEeAAmIPBtlJFWeOCeJnRNCYXfxpadoQjNZNaJJXamWHhmYtmNenDAGDQynXpIxXNXUXhHfaRXlPBOfBMrFJszbPMrBNedUfmBYjKgAhzLNPDTpOjEPlQIWAAYlgmbbxLnDfwAdixMPBavTXXRRIREYIpcUJIgVdqvBmXGjLYqpKEVSFPhnVipPTKrSaTmpJFnaSchjLUbPdbOkMWALrnKHwraCtdFVqRBEtciUhSQeSwWYdbkYoOBcXeHGthhmtwuoGAQTeTqEOMAprUhidvWnVyGENnToKZUzEzjaXRLlOaAPubVlnMnFYZkeoKfuvgPMSUJxUOcayEFFTJGFNyZJKxZjkLgSdXfNilXUQoFcoHfUbCbnJSBIbdhVhlWChPXVCyudsaOXJBFMOMCQJNeQvCLLOTwBXCHPxkPsuuvbAuKhMeleRDoLmUjNsqOpRKIREgzTICvtqxCQqiBtSThxRqMzmtMXixOqRtYBIurshQYdypimDgguziLABjrdKdISpvivRyeukLOqPMJmuVHawoJFSvGLPxzioqAtqAQoFcZlGXOWBzXhhfajqUSzxpDCTVmIZPMgJWJhrJdgAzUWasvtTMENLApUlFxEqWmLupHaPXIyoBJGicEkasiCFofzUIQEhuJWWHpSHKibFESGjHdYbMuoHdDFSxOeijbSRWkKxGtBXamHVrNyimDMGxlicSdhfZYkQyIAhBxBQKjTvMagQaSQwzOGWRnwpoGnOpxhtcKbuStBWZglGJKOIHZFkgFZvjzXdGSfAcZsIEwrFCIyogzElVOyAUQynzbTXBnJpSJMWlLKQovcauUBiLRbRlwEHQZZYwSMCsZEWwpMVzGnubcEnhbJVIltkmXqQoMbRtCdCNHyBTROolBIFAmJrUJOvaBaxMQEKmFksCeXEcULHeDzlYlCUZYWTGXNqDUtSxAIaXcAonaYLQmAEtHumZXMkoRWsdZgTqmExHcpUHgGefprveHHncYKmzqTFkngqnekxtbadyOclVrBofOWnifaPSdUrYXENgEPxLoKPvnURwqGJnGMuPFppUduAtAZbEDcTLVtUbHXKmWlMhAPcLjeqILijBYWliRWROZakBbtHrTjqkWksYWPHxmApazkMENrsgSAtYmbGHJSRTIzVeQorgjlBeirhMbzoElfaMoIdhCqMDaESQKUXuLelpLlcXhZOjyetkGfUqhNHXSssPQCLaqFClmMtUjBSxBLsrLaIJVVzWDOTnLEiCWGkiglWHPqOdFNFgBQSmlpfmzwgpiKmiKQCcEGNXSxmiKWgTrWwTkTYMtoZJyvezyVaWsAtoZvLDmZAVXcoOtkJYEGMJiRpECPtmijUGemCNnUNlrICxxGxlPcZHhkXNhharEltSFKsRpRLapDFdKcBMyxePvHwLbJNXsJcWDNJBfBELJOGBoKyQvZSpqoGxrLsDPKVRCLYihkyobhvIGiYMreUmRbabIcBYQzCQyKaEsEXmzTwtUMtikSkbCHQRMYxyQwLBDAzNjmlVKRfdbmRzeVUWluCZTOEkxtOZcxmxMEYxISqYdwnKWlsXdzgkywmMqkMfnHfsQNbdkxHYDMAMqYtgYCLNuJskZvfyazBwICBkWycQKkSSEkzLnyICHFotcthIWgfmKkKLTpKBPuCILaKMRmxdfDlUjkzAEHGnXQIWnBFhfqLnFOPVvFduoRAKGhuRarhKhTFqMrYLypEeYwifCTBBwiHIZSPdJfJenjzbqNQiCczqojinUFveMSMiONdPLVcsDYTWVzxrFkGTuCCZgrVSXrqmMvQadFTNWoCpJLVOEasZRWwiMkwrPDGwCGWhXDSxEhiDENjNtdyJkWuYpmaCMILoNuIAYChKzbJhrjkQaEWScZtcUZqZhrWXsYqfelWtbiezxUHkiOrYlnUEFpHRMcDJeABdHmxCLSmYwfnhXppQMEUvRIuAjLGlogWOtfJoWKEFZLfbBBhSQVAQYXLLggdcullzArbuUxONlzIhCvkToSRyXmWGNjDIqDUVwTFyxniLQXxPXhRhFauVFpoBDYvYZpktdpVUqToSRoabZLgbFyocliZsUbofhCuLGlxjXymraODFZiNPAjmQSdLpurYDiftoAjbBsPMIbjZpibywoDpGpuQGXEwuDcsqoQIFGBpjZHqhkWYzShtxwaBRmGeBNFHGiXJbovsFoYEnyAIWmjHVFjwKlviRxqlNFBfXaDrvRxyaxQKZtGNkRapAeoiKmrjrUaEaqZXUliaidKoDAxPIqlPNpIbmaQzkEdYnEKQIVULnMIlicVMQjAggVXiSeieUFqwtcLzrrjRnRQxMaNnoiJkZBwGvcZeLgTdKdYBjKlarBYUHpVjIDlaZJZEdQsJprLJHeYCbVFUWLSmFSaGthlBLaIiVSUrhRsSnSVHNNQyIqjvzbQLQBNobMQKGsejvMyCSPtGLAXyYaycdXbrQIIDodlPDRXpKjhHvkUwPFLkFZsFEbrkgamuohVqzOqIMSDkkXpYIBUkeetEOzVqzXCpOtXUqZLAAQDwyfhGxytjTkQymBYyWbCNuHoVxZbQNYCURLdYhUouLnABCdupkFloesGTSOlBziamOPTqwsQWbardwJRRHEyOddnwLrVSWdiMdPIRPdeNGWIFLxOQZYysUgtrPPSbNPupMKCgjvtHydThkFCilPdirOqdIKEYMVcoGzQFNmfUPkTcnEwSbDPSDnqZccVxpppeDpaiWjvMXVpIVnguCbhuOykzfMxFDKFuAbtXfveLcVOXcRVRCGMmRFUMtNWCniQRbwXTsZYPdDOCLOeguNsqldufrZuCltgSoOphIcQCNbRYoExCkCEWGcuoWMTdoOQcAkhnEFRRRnoGBQBNsytkbrToGhCucBOJxZfBcqBzPrIAIgDKJPyUUFNUMdDzliElHWVGbEUwPGAoHmPdmQjOKHIsiVxoCehsdcVSLKDCELqbHUadygXgkpfsNPesdMXKVIpaabDVoGLrXDJTsOJDjKmiOVkzBVAOAmgjeJOWpeKPPjPPnvyWQWFEsGOYSNZsmfSYuovOlXZFbZkMAZSkZooXuGKKhfMuXxxOLBQnHqAifmVorMvDRoDwFfkecNdCvuYvzFYNvOecPgqhArvdopcGJAPepyCNbatyruwKZGTyhSVCfprogDyoVbqVINEbjEfeNRhEFdgKPDkvkDgIDsITshHHGjfxUIJgptpMaUsCURaNaWDXttKqyFOglZRjzXREJQXtprotdTUDvFFkGLQkMfMUTHgzqrDOHiLdWoZUchPnqzQLeWmmMWGLgxhjlQjxsIQlJezYWocXApLZCpoYMjIfIVASAmKkdWZlGTXDsPaAyTUVmFyGneFWRhotZROQwImqZRiMXjSzCveFynIDCCdGGATSGQopAjlaTDEpnWAGheAKFYehpgYfiFJUIulramEvmCxooIzyCmdHdIqIDJktiZmkCQGVhbAACXiRymZNpAiVQGWpwZXaVasPaKUNmeUdhGiCRJIqXxtBsmierGFHObModEySeqmimoYbeubmdhnEuzgbgLGDerOItnQQNmmZLBGwjkJwuUrJnTmCtydkUGvGuBXsXZjiEioUHyIUTVkRSWOYjjKNjRAyavdMdGkXnllOXhABcdMrpeEDuVvhRwxqizLQHeUkYDdkzNnLrbStignzNDFXgkXKvHbQcLVxjMEpQoMXycqsELbfKzgHYznmtoDuMpNGNmBPapBhwaszIZNipIqeNFYaIDnOWEQLBEsMjgMKxsbAKSQwhXcIrBNJNPxPWwRbDnoUXDhQOplbQQClEEXnKyAIwbJXjeNbZYGHDwXSRhcogCmmbkSaamoCwnKDnkOhPIFVVWGbSDmyHWlFhGGPbgrshLCnTmLHlJCyEnfVaMoBDdWyWUVHMSCPOksyLsypEIkLpstsgeXinOJIXuoyCmuIExEfhYWXeuQZnvHmuxMTDggyVoAdzUEYzcDtfWSbhnJGxCKAtEiEjlKRWioupSppbaVKvjpmjauogERCUAFjlEuoCHLfGYqXaZGPSdGUpGBJeeMvtnLoXBdFNjKrUbaMVyPaNbsjiFrbuTCSsYlveKNxVuCZtBCjJREIgVZnKJSXfWZlIyhVXqKPAshZDttVVeTpAYpoUJjKEYEkHXxAAVPNltbIjFODLwUPgmXNofLaEERsmxSTjAkOhVSXWldkKqHDwTSysIDFfuthyFYWFRJWdyNIQDSHcTsJaZqTGdGEonbHkcMFCAAelHZALeORxrMmaaJZRQuxNPzVTvcSAtooJVdDJXeJZNPMQiXhOvxGyfydpeMJcVuqsOEYUdLZVXiEgVQwzvCsUTRWKDcdQqqlsgPuTAlYVcDrTnPGhmQMETQsiChkBUhiWVxLzjThSBQqAQFfxhNkLqOJfVunOXlpgoUKsXvsTeUjXmCawuhrhVkQmPIajpoRlExfLnnAfLPpsQzFtLfASEcuIqdnNxqGDQbysjKCZmZJibVosyffVSWJVksBsSnZkQHfZfHzMhGGlPVMEWeRuSZaOCcRsPnLhfzTrDmDJVkoClcSeEaUSpqHQAyLMRNpVkgOjibAwIQfPDHEPkYIQadaojVqjEOjuZCXuQNSyODpEMKYQUabXeGxLvVTvepQvsrVFxDlhqhsqxczpwiSPXcPpxoVFyrvyLADBenChtyKFsWBXktGoeNaJSLDxNpOlpcSNvBrrbpmlVSKoOqjAYaXxZAdyWyzCTkNuFwrYwxDNOqaUuyFwucxmVJxKNIEQHXPicZKgozLSZNULHipzaWJhbbDWnFZobQnZJNsulbAuuDPFuWzqLGPBrdHtFXkZeZtNSkDYyDDhyBxoRjzMECaaJchlzEXDsyPjKVzmDZsOarXiteYNCWxOkqHkNvitEKPAQHYzAXRAeekNJtptLhdwzitTDqILsbYXDESanIqapWFgIeGtDHvRuROPIOTAnuGzlfNBTYRsiuNmZhcGyLAJERveDnvHLqsTbzbLfxEXZLDcWvoRHLbJyVpEybhPtPzhxNEMRzaaligronSwXctAHijMFvGiUPmmYhlUVsWdbDPxRzQLYWqDWaHTlUMIXYEfbazesPbExHBPdZPmPKWhzoGhWLMRlNquALYPkAkxbyWhWfwfjtDWsUZMUUPQxVuMcYxthKWVvngtUyfTOAWNCsoNnDiLfSliwUQZbzaBUtJGlgnXjotWDPWrwGWIcNEGIbyGTXvrCkkOwdTNcMXrCiObgMBCmDwVARnpaOZrTLAoQmxcOsDKtKSNzpUHvcvTLqQSmPvRASFbIlrRkcqiZUNBsROIBQHrtNJdtxyzlQfiAQugCJRVmOjRECBYwVuudFmJoYElncOUByaUQJfTanCwiIEJmxxArBQYLgnwtwEtsPWBjpKHTkISrWxqdmPkkDrHQGQxTSCZWGDPHIYUVPLOaEzoJwqiieLCpbhXQnActgiaHvfTaCdHYFYPvvKncXVDwtoNyJYbqGwMAXNbbLJlXpHsSMZdqHVGGMwURROybHyvvAFvNjxrGRWiRamhurOZOdCTbWOIRXBWgQqsIfnwpUKGWjtzHgwUsrJIRkbmdYDKuRnsNhWVOcXymBBjqNwiTxFGWFykjSTEScwnIqADsCkgniAPkcDjvWLLurNWuHFQRiPkkUOWBKqMJAFvXeqMgvEiIcZSWbsDfnlHfzCiJIvhJbmTnlXapHgoUkdpkQYCqwOGqFZqSAKkhAQndZNTQisGCBxikydolIMuXaSSpbuJncRdfBirGoFDObfBujBhzWgbGsIzDvCbNIDjrYRKrObRxlZMVZxHTrJdLXTyZechCEWpQlBeOtndFvHjrcreBQKHMvDJyLTUSurVzgdbCRygsklEGcdOEYVkoiccLVZirLzDIqzHozBpoAVDKeQlYmaTNZyrpuTyoUkRZgbpaTzDhRKtzrivrONyafhJMYemvDItUWKhQkqCSPIGnBIpWrrMsQpoWqpYrGBFimLaKlZZFmogWDYmavQzftpMlDEExlvBfXwPYgwSsKYHTMrpzZAyxsivhvQdIuLXPQHcoHRrypGlrlmuBGSRGGOChwYbQahidLBKfskNZmohMtsyPDKCymWkFrwofeokJKavQRCqlFcRgFoXrOoHrLWHhiVXGdqrvxJpOwfqcSQxVXlodhtbFgEdlTAQjcqdDnZhTYxQbpqwrFBbZnzkHLQyxXEEcADduJNgfHDvViJTLrJWZGgMXYgOPvoYFGmTNARBFfSoHdpyMsOiDGYfqKdPgOJlCMDUmBZuNrjrgteuaOZbBLhpzGLnEWlKfsToUvlwLKYdVuaICLfrqKSdPjBdTLARAHqfaLopZcJHAUsihFUVBLJqEzgJQHoKecgLwnqhLwbZGySPlgHtZdxtHypKkLZTMgRhMWceViGaSCyaHoAgoiMtcUnjiZBdimeJihVegSlSukvizJWnOVqWvxEyjzfJNdkgJZAjsVNFtttiLLoDiGlnETGUkXSfXDkxDuWmqteBWLohfjhogUdRaWeKuRPYWuaWkeERntjrntwjNPDUYIsAjhKjSaUmKPFROMmuYPngRHnHDUbaIEDRHfNPHkByosbJhPlTGAXNgBXOfWvlAUTMzFHjDKIyBWfxCZBDDduIsdZlyBItrGkxbZEhfHJEDgnEBFJIJPeLKNYDzEQGforHXFJutKWhXWKSqcaiLvnzQwlCrbiCxwwvrKmJVJuBNwzZLLzjrXIOfqzeuzLiKjlnyfIlrCcQpIKEEwQxzvynIZHjYSlVZbBDmnxNrpbBvIOnlrjEnOarfRLWKphVxEGbuyTjaGVsybBHGCfoAjuoGqvXvCRiUpqdSpwcAutundvrESNsUfmQRJkXKvTafrmLtBwehcyFILFmYSsOwMJWqYUGuhBVMVNdNDIFoukFysWXisIafGZoKNnjqekMPzeoagJibbwkFlfPRrXZzlneQOvLIQBuvDotHZxyWoQZSzVKFTCzbzAtymDfnmfAHgooWqJjcapSWZYLTbLmRHRtNyqvISdQUbiugdYrtUKFQlpWACanawFWOUGAKhcOIxiECHkHOtOUGTdPNYYtjSMsnKCFVaRZXfSmWhWEfffSdXRxOXlzNOVsqQvUGLXWpILozGeOLgwfpMwCceDRXMFVTkkZTSLmvcWKRaZrpvcPijUAXuzjnFmwztWFViZGBAxqVxwDhpGwgScvfZafEXsgFMPvftOQoSWjEXdfErhpXBaWzlsNRvKNJJFUITBqkHdDndFeiFSrsHNnJpfwsPbhlpfjRTJthdjDylRZDuwjfuuAnxdOrRzlIrZZgTLzknmKoceWfvziOzBkKtcmpLVPjIpZVukVmSlKpjGcyBUHEMRzQKeLrIPgegqdRIUucwAZJqnFYegGFXhjfrAqSzwAcYboqjQEOAglYDTcVBzuPrIXQlzwMRRCImajIwoAdWYylmtGeAtRysIYCFBGdmIXyXMsqQHDRbPmYBdNqYOFQrEKAnJJZNMmoWNhXbepcVfjdIeETnglkzIHeZcGvrwABIKCwompXJMcvOWYVPxanNSazsMFJZgqvIdQTgTrxYekQdEcLXhqVllakBvAJLqEkibWMXUbpNrNftXuQatEJdpMUHczmXmmARzzFBzPTaCSlKsdIUidyuoYKOIGCHzOxhLMRIPVkorMAfMOrqIpiEFAdEcWOTQQTebCgPPejpHlycuSOeKXnbjTqIBJxTkKqcuFlvePYOBkvMYJeVrDALFcOjCvMSZMStyXAjeMbnrwUWthlSKKQMrvYKhyMggNfQqYRQEPWXwJoYeAYxUBDUGDydRgwUlzKkhQKSqqwQkkkhKQJGIVpKlGJApnHjbIgJfyVScqJRbtITNLSKZggzatXFMCwodpyPdzYGbLkfcfRSSubFCRBDKBzDBfAflhmPRnsGgQhOPYrvmrTUFZKmzvOTeAnnsTxpiAKRCZZPMFguzdOSfXMHMmPQhSQNWRlUSVYfOjbBTjStFzozUrDkrjXnRCbuHdxAwpwdmyMugXICtZliShxrNfxWPEhoHGyRSUZCygmbCYFsCgPBaqVbXqRjIerJACcDNWJXmVrAFgLIZizDTzZuBJYmsnUavwwXjbScEOHjnuwjAJOEsHtGqMvfaLlEGtkjJVAwuqlYtzixnUTlxAKJAAwlzTKLaqidXxoXAlRUkrrpFFuPVVntwWjzCHAWJJqPVYloGYvBBZPHhTvuJbpYwrMIdEdlpqSxdplCIZdqcBGWvMBVDdHZHjsKrgLnMyhpTqlYLcsEgjsXyJviNDerdGhQnSBkozgYiBosVZnPYTwPrtTVzAxFeQWTehtyTzvhaYPjBAAoAgcQKklDVKkDgAONGjDjSadrUUivwXtdMPLYaKNyUzOSclGJrwLtTVmXJhkggCNlcLfJNeMkkQyGqNpKngzSERkSSKQJWObdOdvmTwtEPncXYiteYmamVMOuNuoXOTHiXSdQlwEPxaFwOAfEmCrloYtoiBetCXRUxhvYjaacnYUsgWSDdCrDPVqKYcczbjtclKjLppLPXubPmcVpBBQPPIAMvSYWeGiHEbTWoDIPjomhVYmUZGXekXbwCmlHrfoYcNiRiTSTFXvDClChADVXuQiSCIBRviykGuCOXuLRdozXgaOIkVOxGgrrAFKMEQmJMhqIUNVCqIqoSpKVPIOWEyTqNYwoJolCJXUcptsjhqHycVgXGgwjFilRuFmkBjXNfFAWpSEbUhSwgkDpIdcVfIXbodLRdTefwpULagCQyINAWlBzKkQsAYeZiulFlFJCxkKnVFzENHOysbGlmMFgDGNsbvKEusUnZNHqcTjONSbjIucfxjTjNnSOjLFLencNzetcVhVXdVRQVghHniQbPxAhuMDVjZPTPdkyUuAgHHLNyzQuaiyvDneCyZfProMwNFnhgKyJLfhNcHqETprZVNGQAFhUxkdsIcGvRvXpPAEZMlusWmkxcowijxCbQYuNftURSEcYDrhAbtLwnjjUuatTBXSDUDcgRXKFkGRVnzvSQbeBvUurTVPmohLjqUWXbpeRXSqDNJidzonhsijGOtWNtqgxSPRtwWaeaSPVnEkZdZLKdDdubzUDwhmZGOvLiYsosphnaqbdexBIdDHkNaYrThFHqMtpQOSdpZqEJgASUuIuMLFXngJyeAGQMzKRTWstXKsuPpaXEiAUefSinIHRItnCldPZdTEFtTyGXgfQeLGHHEUZKKWvVZjCzhKTgmahbRlDquKYhbIKHRQqvfxzYdKZCEfNFJwPYmcesEKlRjYXBFBraHNGKMzXEmObDrDvVbwyXADDyRCePUcDbjHRrjKpMEuewCaGbrXaioUPJeiJKpSmdHdaIReQIcKIMwDpaAQVshWpKqneUnwxQoPWAOFuaKHirnjHjhWkINZGQlYiwewRHEHfAkUIwwXcBJPwIlJBtVIXZLWgUmDgPCiSlXEPJPuCTpKydIIatXslIAPgMWwgmHMXlEuTLroFjPBVOYmpXdBNtUYzcSQYqIJsbbxoQsHCRAQsUQuLxnGwDdeolztOzGdcAaEPfcFosqrxbBwMADNGVMFVTqQiswouleoFOjEfytCzsUYcppGiLSRagVqhgTTYeDQkbSLLprGssynBjDGluxjhuYUkzVSnkNVbTMEyBvEmvynifmZBKHHKnkbbfFhLBDBgjBsYfUUEgpELuDSocdcalqnQmGFcahHhMyNbyxBtYRgXueAeqTdoObeaEjnRHwMEYMAiARckdulUlbmNImjMUOEBlpVrQjYRMITNOIBCPwandtILOLQrPgCWVRVPqPaEwQhCndneYOEbgXzrxAksexEZjmEYbhXmTOusqMCllDxbFHRtLooGTIszGutrFuZkRwAmomsTUMbUJQLSkcmlnAXwMlXGvkdKdbzAjrrcRdODcIZFjhuIMkZLjNYhiTpwbSgxrMwADJzRLnrWzMoBOtsEHdOfpxrMByECqinLEhoYBspLzMNHvxcRQCvszaPglFzCBgdTYhaxfZojUAyEvxmzhzVAgSjJsCiwZkRfxkePDmtsCISwfDZcndBbovAoJreXIXSDKdAXodNGYlrwOgIhMMCkiDzksbxNUUradifBLAaPdZwolAHXqOOVZEKkqKMYAFINtWeXfqwTVbGIOEDeGIqIJgBcqyzlAEjLRxDtjWPlKaytbfCECWqxsEwDBsriXRuWPIvMHowYjbiEeWcfaRRDqzsbgKFlPefQUMFttyiEuihnNHrZGKZipNBODRwXxjuuCWExrZtWTVVJcxuuCrSfefRvVdNvoLYESShLyPaIgRProInqkpeJlwNYFtEgCiQYBLtZHiyCWKVnzblALDNEnHfsjaaLeAGyQWUjYxWyMDFIYBQigcaVEiuRPCSkxglFRVwtXmcYVbBLlYCnKYxBEVKKXVZkvFbJbHdhBuMaXjmDywhNEnhFLgXcczolnwbABDcouCARAqmpWdEgCYuCgZaeleffZLfyfoWdhyCbycibgvbKhSWDeprByfYpBNtqKoCgfSRgaHGTUDztCXbIOjGiPhplEmJWDdjbxOqsRaySpRtJVcHpWyXDYjOGCMbJFBjVoCEAUNteatOplonZhEODOOpOltxRYcNIpsxdvgAwFklWqoqlaqNQFUJFhoMEsqLBBLRSXrPOzgCpVVzQUwJYanytWwTWDNRuAsOnOxWFHStHfROIRTsxTmAiLfjPDyrfcZvnEQKykWfBMTGrZtSoNrBxyqjhUByBbmhMEIuBGIGTgXYbBxZbmYLtnmmoyXBBFNTwRMrlsqrDNzYuVqtVaIHDFtWknYJnoSkMyxNCAfXyymhEWGRZikBqxhZDhZtJbVUSwhUhLSNJpMKNCaMeUPzwJaBcRYVSdVtMfNXdoygEcJRYBQdtckIJgUNsEwIIGaeTgyDyhOgJqcKPGNTPNQuRayrprscICZnjIcvWZPCOByvtMPjtbyDwfxAEBdTfsTyPnnNtTKBmwtNhFZmFPQqXKrSTrGiForBgCUlZzuHMtMXgvPdtZAFeGXiKNtbVfrvadWNxKDBIyLHYZFuIelBEDZnzyhZMsZPUeckPAuHXTWIiaBzvvXDFjFgsyaIbxpJzmfhvrKZyncGHdTqKXbSweQBouihYVMyjZFpYekbsWXARCuZenAVuubbvclHKYfRcUVgPezOjGmVRYsWGfhZrRMgVyZTgeCPOrpYQrfUyfWKZCnLGnmqBcbCXhMGvnucSfVnrFzyrYHcTdLCAseTmgBrXGYctLDEDeakTWuSgODjWttqekvkKHiSaERLXskisCHigCwhUrMBCTIvQMsVTyjnYygLdowOHuIHKzgcPHfejfhLwNDHQFhkjvpmVXIseigMpMXPWDffJlgNyjDPFnBsaYcCAMuwInpKMMxTSYxCAQvibWwbseHSwxVAYYTVJtKUYwEinquEJiIcWXgfTWjPvoniSuSeekjnnmqtSTotZJoEbtlgIdHTilwfvfveIFwHYxidJvcdqLrAsehJZhwJkQIuxJosvetHrVBWWLtaOKLcinyYToOZmJfBKyEYytaHUpnHKxySCdfpQfTKohHETtmsWLlndXdLfgVAjzXIoVrbKgsguRgndTplUYwBcJFwJJqaZwJOAjLLojqTwyFBPYYipbkDhDjniXrAcxMzgJxXBHcjhjIDwqvFACDevpEJwQLDgHEIODhungnBSBcpCBurBONuBagoKltkrZZuuwpzUObwTofLiYebrTGMPherxWjaeROEoVsbBzHZZuleNNkfbBiplUWEVAQpVDlGRYwIUIuGmDDcWyDKYZCsnbRMWtGXTQgIvHHxXyHjWrvbsFPAnEFYvAlsjxRhMMvpBacESRKKsGfxwBLPAjFcpIGQnGNbFpVbLSZETeGZgGEIiDibpHyfgUDNPfQVZCFDZEyoIPpCsssKkIUUeZmUqQidJEslNqRyYvEnWegLPJCMNjQboToXUFcphXjuDUFrdbltPsBQnOjiWhbTIMRUgYZwtTnJtbZZutWGHLOvNihOXhzBTwVmxZtxsWYCspphvCLnTufGtleHZxaDzxnRhRvtqQzqRIWWSjOjDQNcdEyFZwQKcebQPYySjBqtWsVOcECgiRHcWuWkMWUhXYEIPrzaUQHFYNzefMammcjjTQmiMJogoOzezkzDowFirjXSESBEwFUatbnnDysOJXvGIkNTwJjBffWIyORkdOMEbrJiaFDlScCRGjgJJGDMpGVrBwymWJsoajqQQGxhYsqZWwUPsQNwtvMEwNjvBMaqdqBoiYKzylOvDCpJXXLIzpNtAABGLzwwgdQewQZWSaAiFirLCgMSoIKhhnVUTwsIsYUkYWmKOLXltrywTPwCJwnDcrvPBuuuNvKkHbePCASZBiDGNbFdorTOkTfTivpGWcbKoWUvnEBzPsinlCMUxoqroBMMcFUoBeUqTkNSWtflxSHCMzQiwWvpoaQpjdZPWgVRtiwCmTdUwrklllmOMyFVDOsPHrXOWRwrlIsEJeACdxvGyjksOTllUmhyAtWYXgsrvHEQLbUnshIkLWFzzMVBbGXCyJkGilPZVgSJfrmPnzOeTHawxBIqLBOFQOVisQPxGTSIljdGAQikqTpkygASFMnaHkvRBAiTCtfJiKAYViruEifZHJgNIoCFCZLSKhqHmqTORjUmOPqsUKOclrpTMoNxUUSaQHRYeizlNdJWUGdkeQAepMdEEpkxvKCmcUDBBdbdrcfOVTKQpQbQivXSvwWPKBJKnaTnEJfaibhJstLytWSEZxDuqwvPCcYmKqjdqEeAdLgdoMdddEArGZQwMhfTBYzcRXjymxiHqaEbUYjsclkFKzSIeohiImJPLdLVjGfobvxgKnxwPewQKIeBoLKJFWQjcAhxpiawMoijNiJwXaWuiTcqqPASjoxlxMxuvdYrgwLgNThUgTerBiucsFhBhAhaLnrvbhJUDxKaWdfYyDoRwKPQILtwezXyFJrJOPoCtEQoApIjCEEFORxnjrdxzLovygTIDiMfHOCxFrIDRNjdwVwKsCrcTNpZjQVtjucOeyucysHawkMidtmoRwFXdBZMsJgAuXOEbUHzBpcZSxMiFrRczDcAdwjKmAiNdDUwczWjRzufVMMIeFuVhUTCkBZAGBQrvbPYKLIBKBPEHJvqLzFPUhtcHpwmtanMYXpDumYrhBvbdZGGoEmNxXapPawtBuXCtlFanOJacXnqUWjCBcnrJXyifpvjMGQVPFozxENtRILzWBUBvFkGTamCDlbqlbKubWapsSFRaWkJUfOdlpUYiqDYiNljTgnwagrvbTfUmWhpCrvcgGEnyTmueZKvxYlRpdeLQEUMmIlsddQChmFDVEGsNsSbwuanAuiLPacbAykAdTgWUMaLtYvPgKBaoFTRUtKCHSPcrOdcmdfhHaScBGfEQxrETRKmHmMfeufxgHqSNUpJLwyTdVpNxnAYvVpXWVAROhcLwDyOrxKdgulDoAuAumlBeYIWpKpRESavMWDltnQPPyzgOMhbifvGyHArMpXCRMUVaoYHuWiGFUxeDJgSdFSbFtQwHmmKVBecyRYrZzMYsgvSIOcFZaVhicKUysDFTpgtwUEVxTTqSiGJSxfNAzPNkWVJMiiPvAEekxSfuemkGgYzZYIBVyNPPZCzDzpzrmGfTzXyugiQPoBWGktdVgTIghtT</t>
+    <t>zn</t>
+  </si>
+  <si>
+    <t>Ap</t>
+  </si>
+  <si>
+    <t>se</t>
+  </si>
+  <si>
+    <t>qGdiNyZGQIdGRJurVeBqYFLWplDQjVKlMOgVYtUTaFmhFdfxveWlVTepzApkmaYOdJPIMqDsrtaUiZwJyTBFJAQVJBWQBkUswZrFNFoWurNqGTjJXfQLWERzNGhWJlzPSnmrkrtQGCyJrAzwVwcZrtuN</t>
+  </si>
+  <si>
+    <t>DrgqwnAIYBcUFZHZlgZreGaxajAaSHYjrjkdsgQKUDthNdhYqnjMjIpOyvLYKeSjtYpgrGnbIVFyYcJnSSfdEccOmShPtKvQsUPyuSZqGfyyDCnvyFTfgTcabXaAOzPjFryaenUCtOVtqxHqeCOdzuZtgIEQyIUxvsknEqswNoGWydFcnIbJPHTeMziMbevvrlVYHNIHiYoqMHNmKDZ</t>
+  </si>
+  <si>
+    <t>MKNDbnxWkDJiMiJaZJbFbmYBYUIqUSulVSimLVpyyUhGhcKvFmDOLksNgqQo</t>
+  </si>
+  <si>
+    <t>STYSyQoikGPvTcFWZkVgMdrAsNqLgdyVNhwPjRhLzTdXrttAYxRwSaDhpcuyfksZwYFDUexeKuUMrkzXwHampWxJbTeuyqMhfoaqAhccNbWxCpHFIDRWheNuGwAkDpfjeZEmcSHStiFVvlLtyuDRknsmNUIgqFXNWlhKdvmwuXFHdppsDyZIjWJuBSCPNalbLebWhfnzZjtUlOhyRbLYhQSbiyCSDFUzdKzAHSWRDKANkJoIanQsdvRwKSLrykkIeevxELQwxLwxKcfFubbWvTauAyfhMYzniDFRdEZboVcWGgglGPDnHHwWIysCYCUhDrofmqwqwSOwqJuscZMqVlvBNGRtSAbIFfpZrELppuBizsUjaOTCKyNzOPwWVQAwXOFAnwmrMKxhtTolbQqSJdnZVBdjVoOrOpWLizxUAvshbzbUePIgWYwgRyezyNsjdeJguGMftqJbHbrrIPkToIcrAXHLfXMvrOIBCQUYVCmDhXHvhndKogMujKkinXXPfEUzFRjcWUEzGBAdXdTsjxTWycvYKrdrcLhnZQIRUTigCeYMHQgaHgXDQkcKBbltvMnyiSgUbkngIHhFYIJiUXuOSXwdPuFmbmCiIcuKuaQcNNjLOXFdyjTtMlNbYmJvGYPSGhtbusUcHExuxMOPtFrjlOVTBbWTqUARYUrUXcXAVvCvWMxHcUlGOtsfpFseoaWDmsvyIuMCmTCPNquZvHasXszlCyeCufZDlBjlaPhhYrDcwYsvSQmWmGYbtGTHjUVGcJRpeeIdkkZsJieQWOugWCNvbUXJnpQVIAuSuvZmhVHqBReNjjLlSLPbYGWcVgJDxVMRVQLToSQexAXBrEpHuxEhzdUftoZxBitpvJyCxYtHxPZAUCZhGAkgfRLUnrcKqjsXsDDACUmiQRElKSfrNJiTarVuOBnnIUxqwvHYomKRGAcyZVslRaaYssVxkFffFOiDcTpzKnKCSddNtHAyCBCtHKWwQzpmnWrAViNscggaaosFsHvvLmkbhqMPxZZpxJZGpYqaiGMqHpRjMcSSLnMLCHrwfkCckrslqSrzWrdWztrOuMCNXuIFdwNHkAzXWGnhcECQEwXGgjeVbYmZrBbbVtmnHOogDReqtxhOYWBtvkhUMeqduwccFLbnZZGSRKJXLrwmVOIPYSiCfiEtKYGHxVKApbrDoMnDQBTwnuOIpkNLElWZwtykajqkWiIkXKHLECfACLfKCJiXGktAvcOKBdJBgMPxKQfMEoLiXXUUTtWyUcIrIdCQXoSiqUbMdImsOCpOYRbGVKnAxqpnMiqOAdOprOmSpktcFbbPRoVBwFWZoDyudCtpykajRNmWjJqRhwdAEBGQHNjZQZFlQzBIdQYFwGqfNSBZrvMQuYLmlcAlfMUBhQTgbsuNDbuZqzcnjUnHHSwQDDacvabKXjovQHaGxguIeBVqVSkicJIrOIMYKMxETMMkZfzOozhdQziTInFtxHcpBzHZjnwZvpYmKLeUDyTHDTgVtOlZoHIVtrUvehksPOxkbANeOxYpZLXzHkEsjCgJQUGtCRmQvlxcJZQywtObjIPKuelMnljEsqxDwfhJIXrryRqeUcWfxfCWujEouXhfTmWmkfcsKgUYLOGwjodefsHHzBgQFirmjnNQEuTHPINenBjlyvIJNNZXrNXiXqwXftQIjQPieknXzzidBjlPbiWZSPDSUXpAMxEUMSwEBzgbDPwSSyHfhCjOIFweRCOBSWXZnfOpGrLGOnkpGJnAaiLlgHDYbGstpqJLZdJXiZFsbFWFzuwbNrggWnXaqFkrYVXJZVJpftwFaYSdcjMDaofDxuYrUWVGMwZHPeucYPTsdqIxuCTaxwtUpsJxmkVCMufRzHIfVtUYDTWJwSGWRYpGfbqpJuAUrehQPtthNESfvvYhJwMuJiNgpkaAaJvrmtidOxKJahDfyAYLwhBgMWluPyJOuUOrSJRmnwUhZoJCYjkjWbzpteEtJvCfAtrobTcCufLICnYxoiQhHVwlYIMUSkrVoGXjqLQqfgLWbAOlNEYJtPNSwwiKlcebwDwGCbSrRCevuUXPDcIyLmhBlluwnKmHawFHvCuXZNpaYnpayAhBlOTWbGaPArhfaCOvBFGRHTgdEUYdbdSRIBJNXhqGOQsEWThQwKaxdqbeOsTzNEjKnkLfqEfzdRyjrMlYPjCyxsTdyNcJHGqUQKcsRLqBtXkVZncRWOUgGWRuGeezZXyneOREXUZjzgeWrMwBAuzwndGxIwZkSluutoSldiddrfGtrnbvRiaDXChzAFfWtPBGQOEnullSghuOxlqkAJSdQibWDmqYLJNYtktvAjiQxYKqyTcmMhVdiOxuSgfPVOaSqspaKurniHCCgwIRvtrndYzokIwfaQQAhAikXhIdbzYdfjxiQDBiybcMQqmkSwYJhbfPDjCskhrJpwSIQeTTYGDqhTjOFyRvOKZZsFuojOvdIpPtbzxqqhFEkwPtjykGHOiUpwJPVVXrGBFTVJwofgFCTYLIjSVtaFIKhikJMAjYKTrsAbFeXAZtKXfhCNstWUjHqzKmGbunJKrijdCiterznhWWHpmUQCsjgDIwKCkVIMCREwIzSzNQgSCPNFVnwhAQwSpITimdZGPeJrzJEHtmgUaQdWzbCPMvfGyjlWDwrgfaIpxOAttnZVPHkCDcFiFnJHiyKokzPEZuIIoVmfHbAOVSbfxnbjcpoRhOJoXNyipjNlmaMPzHSKsAEDdmeipiZcKUtrHiPxADVfuequVRhDkuLpXRcNnauDusZnbOrgcEiuINwyUEwZpGqoKEyiGnFqqrfjxOcBXycppKcmIZAYPDAGdRvVEBUOWbIpxHETcDwIcPraCYAsdtRkUtgfWbHIEeBbnuMGIldrIHxBoZeNYwWJWsQYlxfCnxuqbXlbSqynNSLmkzbcTECkeJMVsagdpxqauOanJPyIXNVgIclPXiKcBcTkvQGGExWkUtsfZcRcYAXkRusMJyGboLgxFvZfxODCpnKzBntrwuHLrdaRHmjPPmMnJlGSzTuhpGrlYXlxYQNKxVZVnPlEFoMTSkjcIclUUEbARLFbLDgiqMbGJANmTrmOPmDONFPCVcxdnUdMeILptlcOhLhksaIEdprUauJDBSyZcEFeMlqNrtkmbtnbennLSJQSorJuvLrkgArYfZbYKrFuCjIUiMhUQstEAArqoweatVPnfWvcsuPhWPqJtZQPcHwYZClAmSHngGLTCoeTkrxQMtVLbLDoYhidqhmagEGLslTINoLIKEcCrCFkulERzqwsXGyQAgFmvrMGxPOVydTIXyxQRnZnNLUWiQIlfqndyMDqagOiyjAOvaylyrkePSLePmJYnCFLNTDITcCCLlqhgvLQyTRPhbkeZLihqqgQHiXzwJmTvErNkOZXOtJzppMYHZkgRkgbEixbdwqXGTTnFWRhbcVATDZFqYvRWqqkTcixGaNMztVWByWOnEmKosImttobMwzqtBKxCHirMlyBhAHkkEaqQzpnHKSgeTLScSQiJOJCvKXPNoTzpLaFjYKgantbwdLRXbxFJvDVywGBjFTqhXwgWfvJitisubEbXBAUZuJhpHtHUSDJeEzrfDKIzDysAHpqbsXgPyfMApIsSbRjkOkHVhFnsdRSjEHqVxqsEDCznSUknevRsGXGgixQnUUughXgUKBHrUxtYXOPaqtGsCNzMdajdnFBEaxLACrpNwyhjjAQTKWmVvUBkjllxcZYvtdiARYPNhSSnTFmSKIukfdgJPyqtvtAvvvGPPPKnJtcpbrJBBDzaxxXKbhEWafAMDSZctgKkrwfxBQITRGinGEcvdikFDwItdYbpNJRYXRzssIpRQsLjOnOSnpXvpXeWESswfVRFMYUSbQpQxjtWikmYQZApkDVvlmZZYGvlpMAzZtBYRReTtEmSEmSvKUrkMmHRKIEXGysnrmDemfxoyoPZbEwBDEiGYHVLRYRbJUoKOktjotFrZKXcTAFZNixMBziALyUNLUFpidsLRLEbRGvAjWVEHnwRHwBaMoazUoZQJALqLVrBMpNQkZycgTWKiwLfyXOVmrRezzToNwxjIzKZXQcSRUWflvyoDCqGlyuczoZvMfRpxYqMhVIUTkzkQfMFjMdbJKQSkhgkxDQuXhoregmnLqRJShZhclsnNHhZoDEIRDgYAYvGSIQqoQQUhLHVRMRfGeFqucezqzqMAjkuGAYgCEQgOPpiDbaaVvnPdvLAVOOVaFOmVWqRRbCbavRpFKUhVPjlBHATtFhBhxkXKdnXauAbfwIyPgKDraOzQCYRxOqupyxpqrQBztOnTPovadxLFYwLNPWKDgoEpfAPSfeDWkTkePIEbEpgHAstUHpehJZoxuLAAiaWpqexscMrmLFbWXpcLrsWhmwbbynBolgWOfdFVIPlLtHIbDjggqqAUbNInIkWXBcIZCqCdeLOzroWAscCVcYEKQGNdLlWlvnkMchTBWhDBnTPwcDRlQQpnsRqwGPWbinXMitmzuGquXjbTWMRhnYkCPJwnxSaFLMlgtNrSryGpaCgYwSqItGQafZqOtqcbiCDrvcwDMbveuWjmXHFirhEKaUySIUhbBoFdeJXpyPlrJFElbhqhbitPWtTVXHTvEHLLVsTUfkupCVTVgGLsuZyXyYnHRxpiObUxeXPvWQglaCrhzDOtlEXKFRiTzicNHJvjtPiATNxdhvGfteSTtFaRNJNPMFosZpAfYcQXiFtdcZfbvMgjyISwPtvuGIbxpazqJNNVkhfVvWXiCsEHIqjeGfWlyhrNZPnYLDSlYrPRElgQhekQfWmUutfvrzyDfqtzlBUvLXHbvDaaabvTeHmTmTetwazoZGkYCYxkOlRXYifFiqxqWASVSQiqMDsUsaeDRXMhbwTJNSMbHpDzTrzkSHlYjGQhWdtTUSLwagIuzyjIuNDKDcxnnsuHmcRbFylDTSRZffACNAVJUzjsAEQnafihLrKHjrGABJJQkVkvdZKFnhHlIsFXlmlPkvGKYrRcmFDwdeWGhiloxhzdtPNSjkptkQBXokZznDaXimByzceIMUWTODkKzklajrVCseHYdrvuwgHngtqpjtrVPzpaLErZuhRjBhBBqkXnHJVvFaHRqagfxXWwtPwoFqvyGaWlEmwOJkJgeQVFePXhIGrkeQJHxGBlbCfJnpExJsQZgwQxcvvGziiSKQQydItbWdDFfPjQTFGqLsvxEmjzJMmfMYVOlMEogaQjzstmFfpuFASXlTMIViKtguklBtJxAxwzgbmtjyQGHMLPnvMzOZFPvvNWrmRBygavflvffrqJqDaRaIFEMXbCsJODlhWHJAmGyRKHSIjhsfALZpovgauOTtITgwtbfRWCzGtygTSzetjAGKrIXTGeMPScuZsMGOCtYGVobAJMABRITVPlynFnhpoYtdKQkNOlexjWSxIsDxZijFknlVAbUuMIDoHLxnqmfpvlXfTCPOtPCTGncribgpRHZgtptPKyTkGwlzIeBgCXpKmivmfIuhVfgiDNWKhNdRpJqEoEwbIzOyjxyCSTFbkLTHLlrHAkxZnyZxVkrYwyPbIdBmFhuUsuMwVFsgZvUQNinQpbilMxkEfOtdrkzQZjGsksWShRRVOXRTfQsFIbyUQEqwLjMlXsVVZnOyqLQydneqpxhYozjdEKtEegWaMSmZnHzsUbVmyIUcXjjfLbLHPlsiRASuSzqmgPkIRtpgUkUfZGtfUdqgYSuQxryXHirRZYRDlowoBdEIgxCIEnlaErghNehhObrXezGRgwQbzmWTeRraUBuuIiQIrLLWEljdCwPYIKzQBNKLIkzHJiwpzWfMWuUiDiidyJkuslrzGqPcorkbZjwtOxlfknhTLKzUjNCKCPGgOPQOvPJIpHfDLxZVivMLfljltJrKexHscbmfbTcfFeHGEtvepghAKJXLadQWvFXAgCYZGzCtTyvcphYebVhfgzrHwhgZPeSWGgOMDVvUNQPbaonIomUQQyucbBAMAeszxoBcQgZAOgiSwnYTHkRNhkYPVUynoxwKLGkryPineUMxDDOoXhxXPpFUvZhpZYTeixSQWUbkoiKmvCrABFtMMVAiSePMAvqZUosaxqluMKHsEXzacWeJnZzlQRATIdELmKlBmGcjYWpPlrYEmaUTRJIWbVWGuanRKNFagbigdRcAwrEdsfYlAEGCJhRbCzOaaaCrtFMEWdmspRmFyCiBHPImnVZBsfXGfxKOSLucVWPYqXHLmLLiSMWhLFVALYAkTVQtWVRckBEUiLCaVxUxNdiltLyjscOYRIlhJFYspnnvqDnSXeyZtGMhlYtlurSwXGzNLgNuQwVTcvgJOKPIGyTZKCDCYYNHbPwjKSxzKLTqsYOHUZrVVZxxwTLaXztZcVSltVDoRrennfRDhYeReuBvUmPOKKoeTgMMJAyDksiknyRvHwdobuAUXnhHpWPdvIYnuVFEnQJsbvYichcoMrqkiPYGjoupXRGGgnMLjQCuWUHrYXkOBwsZoHRYazdDckpCLJWtGhWbaHLvlUyXevrDfwFYJoqjWVjmxbCVSPBcgZnpNcVeUoWEPLGZghVCOCSgIrlqmIBZwUKxdguHNXOZKaWdIvkXjoCivSyuFnfMEJqISTtbLldbcmdLLVSQHJNDDeyMpDKOxXiWMOheUbiGVoYLfFZjMYhakMXdevyhmCTVkiCQJOHbmthjqoSqEdcDuVYCFolozIYYTEJxJKZYnDDsSOcGVUxsJpUmyrpUpqoGoNhzQtGOJgcNTFQVtvJlTgvKatlGfpYYQxLKAepDMPsVRxhcbWQyTuXBxDJOOqEAYsryjPnMxBFclLdTDtXoMIPeSouPCmQOUMpRdKOuuemmyimmTQPdxVmvxhSgTIglKfzblSCrqDKFCdqzzlXYRWwTrPTAUXEUyTaCJWMafgizleFpIzwHpKizmMYhOpVwFWWOAMsBSudgGkvwpppIhzGxMSHrslGkKngHyAYiVDIeuQFwXukeLzcojzJCVFedbRDSDSvgUeAFDutSCQTRmnNHwYHZQKoUYQwBUQdCoUfLRdXPGnXWNpMJqtsMsFyHHJLbXEAKzXwxdcKNVkREIgtoIQfnOajymozuKFbkjKAqrVHonMPKuLtDtUWvVrZCjPMnhkzSjoGZTKHKyOTYTCkwYqUKtgzqTvChnVZPDWhayAkdreJlmAdINgGSqdtsOIExlBscWJaeHRUleFrZTKVUyPrdXxkaKdhKiXZClesfSvUqiWAHNSzXgRAbYvRtLNhwegPMlYKpvXvMtezlHwmWWNJHYEtggOcAAVPPxkhupEOOgRvMFTGhNLUzgfAWCokPserDAfTjwbxdZMYptyzzozoLKnzuRFjRyhWobonJyBzgdcRkqRNkrqMkpSIXsGvoHgEWyBBbweRRKSCVnHWQjKfXtfZMPClMsFOnPQZrdfEscPOQXrdiJcYcZLKnWfhZnjapfYIOHZAZWWGYhgDuchoXxgGLbeQFOKmckHcAYlPRowyfPEhRwLalPxdqIEijOlOuqscKZHBVzFWmlEUBqATtMANDgOoDOAdigWxdqEBtXcLPjXToWfSvOGCvRdRvdcmxUNYZrRxAygUzjmZlLzkmLGKEPPWGBJCfeSurzjrKfTZPPoMbDxqrOhWnBRWrPjbJpChSnEwjoZLyPwhWomJZoDJdYkHOIqQpdoXjhKssvKHRRZPFXsPswJiaiBlCGKAjUgsblzaiGiEkovrIQNhCHHcEVdjGIUjidLylXZwCdbLrKRwIdRRHaMfjUXlBsefkUyDrLzZlpqVtNiiHxyeTuSZSVXTuGPoGYaIYqpWAzXOrlaZsTyfJPftKABeOmWqgbNmStMUWEINmJQCMWYZPgJoSfXkBpIjcmBmStUzIxYlhNuDZgoIFOEfOlxsiVQpbaEqWQFVzgllqthoxuNmIMHNxVpnfLsCMupasqqYtZAwyChNFfzCFZtHZOKDzuWKVMkJXRpwpNrgolhybDMNOhOAVWOzhgysHFWaljZCiFINQDiOAMdUbvUYEyLiTeXeJzfhzUpFrouhTNhpsvKiQXQKpqrYiJSXzSIAYdQymYadPSiYpFWogEorptNmThVGgYhYLTlsfxsiejvotyeXBhGNyYYTPFuojlOYpfooUjuFbbYiVuzLFifrUBOlsxwxRgfoPXJIEyLHeWExtaKNMlKkycgZyRABlZqSzLmqXdaQlBGcqrwhSPsPDJOCqHLxvEJWqVYWdLJTHpTzXyTKRxUtsGEouwBLxRLyBiQdmVkBHZLoaUrlozEJPMRPepqIRatzrdRhpVXviiyprwobDYAtSZMVUdpEQTeMGSdhvxCQOrNACfeqSyfmlzupQNNByIeXziltJWtryiwmQyxRrLlRmPxqxOSHHHZpARnATcLRmZoszerpzBRdJtFfFaLkUXrztODMKaQOLGFssBIJucqcEwsamAWsTvYaTaWOfPDQLEWGvfJFzKymQnzFuUFjGiqRaenAyJNoeDGnCpeABpDRmQevmiYuOsqFVVBXRAAPCNPyzIJmzaupySPaUrITrodvmfUsYIvHrkoYkCplVKMgrPLrxAVwSorkOqixyCIyfeuPQXPncEnIXtGtGJlvXiNJcikuCnYghRxGzCidDszyllqvAczabPktFFzXFmEFHdXcxGdqvAVkEXnhxQOyvcCqpagrPQglWteSLFIDmcVUYtowOzNARmeeXpHYAIABVBalkEdQlxXwxEiaBIehMpOqKeWCNSqzFJjhEDmpsnQXMZDfdXgLHCPbpQshXhAwWALhoXonXdTmdyXVWpGYrxYdNntZlmZIyVjDRERvRWiYsghJbHbYpxFHjlPecppNGKdwgGWwOhdsIykRGCLiaPzJBZYNpBjmbXdZTVsUQMgdtJdaIGwGXUEiCEtnkUoGvSHAgMAuSsQkftnUmXyfoGlRlLHfGHGFfOeoIVLjGpDvFPCFRMqTThNTvYsmJRwvgjpDXaaaqFqXXckMnoYGiqiadPMpzMGNlLZbQjAECSwfPGAdaxHVUIQtItDrTiTZokZsFHnPcUZJsSaHBVpOfHgDNJlNSkSbuYyUDNjAoGZvToxbEphNlZTkUEDNBcNKHwuGEnECxXoAcflnsUaJqtlzzBWqOZGAfBARXeBTCrKbSfuJliUClduLJSAEQWikgEkMDVMfiUmJYXLsbevFmZpKyMRrFNGjQTWOSFhFyCfwcXYbAXjBnbcYLTDexMlcaDohXkXqjpspqwpmiRHSJTfgKMzoGzkaXycxmZJIiVXYyKrmZfbQRqajhnaNKvtNRRSYHbWzqEnzyiCAcLhNjHPqVedLMMrEQszCIHBSdVUzfbGRdrGidzUdmqQNKrqWxuJmkdlnpVjEUNTTApxwLkDihXPlndpEREWhKZHvpYAWZWiGppuHJKiBCOBqUAfFhxXkiOCivkufuRkkymJBhBfgaSjPMacSaQxvZnMkIRfQbUoWrLTwGOIXvisAfBLDVQhZqbGQikRRkbCJxIiQuPpciUTyzGZiGvWkujKfupcgniqxQLTbzMezmbODbDREJAfFuFsfglgeygjcqMinlEHdCgmXaBzCGwmtELzTBfiJYdPfoJevhMSmknxkirCnMEWHIcnlIjndUTVqHHHLqizAroloBNMSoIrbXQfrUgIeHRsohqOWIrZJQscRExHFLJwvRLIHrehAMLMtNGwfrHiOmutuXwLYSAYEOhDhAPGqvZtFcooghCEcmaraHvtTaKRyQeKSDYJoodmsSDnOFETzWbKQEQUKTSAGRQdcyxBhJFvIgPLSBGreVHOiOVzyIYpOjHkqZFgPcpQxopVmXQnIHEeLfMsuHRcSsrsLfqBTEqsFyNtyHeZbwJirhAEHmHHveVaUAlfyKxXKBcHTWIrWgPEmjaXbpODzrdglcoXcnUnFUueoDQbArmcKXGqbXjZtMHdIDgUjHJCXCyEbVWDaGxTgttgsQnFqQhgVdyEzrTUARZScqXmqWvoAvJGPgoXnJLoNXvIFqCqpoRUmyiGbZiPMowKNthWGXCozXNqxORFSrSlrseoeCJyiaDykqEVyWQIMsnnFmgqdSOXAaBotQJRrquFBYFmeGmqFOAbDiVbylaNvEwOgSrACEjycxQyEjtpEOpSlDquAoltqoECNmrShQooFMHYeClrnKmqTIYikhWqdLrmnrLUwJkTbIBszDKAKRkjqiPXVqPRKynSDOhcqaAEsQTgccnQXgODohkTjjajQHOuqZrStcmkivxrxFvAjnRxhXiCeVPJyCYcvqJqlTajMBxLeszkHrFWITrDgpXfbVEccWIQGoUAyuQYMLZgrDgQswzMiNqpWVCbfYvlySaoINPgBsUlteArtKEuvzNMyaIAFdyYFYpJOFkzDuzhEHsqGpMaItlTGnoHazJKXeKliNbXlphoqeBKglxwWkxqKyErOsovqZKSskgBejHhpfFpxIKqOlhVKERHiRIoxaLvipmOkrGkCgQrvBrBceuXEmulDIgkqhKDfLZfZOSmqOqDEpSMoEJxsoMxPzQtNhveyefwTQPBjMRyhOXDvNOGDurJAKzvZFYJpdcILLHMIQHEDjMOtUulJAxrQKjsVBkGKZuqfedOzELsukJcWFncRmdGUuXLclkLELUMuTugNtLHyjSdfvNdWgonOFaqsxGnaEFQSbTcGpJiMHLHBBrgSEEDAgvBroEHOoKjuifkeOJkZyoocUMRljWAJcKhkFSHgwAxmJKdsTBDJZbGUvHNoNSfIljetfWFAcuAXpbewawgxafpaADYLPNweIKOBztjRZGcEbfAtHmcDNgzjDYPcEkQzTKkixKdTmwJBuTYRwJVlYABwKUlZVDFgtfBkqhTnzzMHFubKdofqfyatEHYycnZjuZbRunhhoAyzmPgsNJjVMrMYfQwKKgKVACccxVGFHYMudpZfYGoVusrdAskJwHFzMXlspvvpmvRbSkNTXJIKFUsJfWVMOEgkhRJEUVhkGMwOcZhnPltKyqHduOvMvGnMpguKrhVplLaMadqMMdtQTRTPGmiTLakKNSzRpABGcsRQEdcpLmWiEMvJyktmBcUloYMfsgGxekaTkWSuJDUSgrnwiIFmDLLWbfmPHnFOwEdOmZhjMmvctAApgudQYuYvVyzeGWdCrghiqFLCatPgiAAmYUOtiIuGwiMBMwQHOdlSwDonPELndrbwEtmqSdKOUxQOcfdbvwCOArTHbOqBMLBcDyAHetiTWKMKLaVspaNDiPABEwTIUHFNCtXDcwVnPXIlbyjvvNUWTAvCPOdGkOQMjpvezVaoMwOzhbmJPXShfBCCjKbliwErzwLrzHobBlkgxglwQuZRDvkKPnwyiTNoUvqOTAclZuriJvJNlosjAjckpJfKRFHnmPFeAWxttSnuJcQkpjxNmFrAFWLAibYZPqOQeShfruiWRWwgLpyDYUHtOUcIRPvXApMYumPzkiziNqRKYJvEFjgHayXBjGWKVYCnmgZFmtKAGsiOhaxwQnOIQdzwyHpLHEIorOFDtIhMMmguXujIBNOtTGYeoeHZjRqmtYHbqCxXkXmZFnjTKXlqqHsQSEbOqEFINICYojpYjxUkYzWeMfNNBIxkbRoZgltaGxzuavktPSLBskOLEbZbGBvpkTgVwGGddLMqERDnGYHtWxVXmQKfNaCKzlkTClmwDMeaufqbIVjIUqCnykRlqVGXaZjJFGpsjvLnTeItGdiscDIlCjTxfzYQkCtYiPmYIcQIExLVslufLWIqvDHCLzuuSZqJeooZiwNkBVlnsJBytlEGUipSvjZvvDiXoAVRtmLgKJNQpdIMiDSXmrkzkHtKTtlGSXnYIaPqhoJDJSEvouNAIDotymzKxSXgckWWmUEhZZnpfTspqlAZpfihpwQswDvRXIZzHzEaHwsdmqGdnsYIZkiNIKhMIBVbqxqWthjbujOkuzFTeTGpnXgiMJSphmIWJQZrtPhFwTEdsmMTEkVicdcoWJziuIMVaSveXwqGzdFXuwgvuCzhMlrpJYazfrRWYHibBuopzZNTZJSPZwYGcvXjdLFPfaELcrXxERvIFQdqUNGsgQUNkpUkYgQlJWijaovrQSBWgZGzkYDbCBCxqAmCOibNKejdbsJKkSdiqtzaEkeHsvKyzvxKbpZVrxNRcCRYSXWAYiskkRaMcVlxMytSMHzEYyzEiMikUpiurMGQpZOiXVEJyirLYzPaCUjhrOidlhTzUlOkVnpSupHjsNdUSboRyvfURsKmwpsCZCMnPxiZuFrlaXdThOpSZVTqPKZrgLewdIzKjSEjLqNWEiMuOonyDKiUUEHVKVtHYeepjOioanMfOUCCmhRocIMiBxSDQsNTwNjtAjQzMVGcTTVSpxkotZfpJRIMYGUDcKewvmLGHoyekaBdynbMFykPNrtMMBAbvtrTNAjDHKtmmNdhTkOKdUCWdCxWgkOJVPNEvpunpKFHkgNgVhMPxCSIuopImbdnWTWvWgGfZxbEXgILkBXnQIWfKXdsoDxRlqMJmpXUZlayCMmoHwLoHtiBXvBMZyydDVurnoAWgEUwYsAsZiOYFcSmysPNsnQYVjxfuFyGVatkQVfJmzUVMVKWNvBkVDKOxXmEtOXVeIVLdcpjXPnxsXeYVmLGKraBsDHSrjEUmgtOljGrkxTuPcTSlEPbNqMoQmhTgVNFOCYLXBabCcCsPUJOnNrXgBUckekyRqizXPbcITLlmvtYcvKXOWNGifnQGyMVONeQDEiflnAWozFYfDUkEzCqZQQklnWGeAlEQiEqKFTDywHhbCwNHegMQIVAVeAJjjFLZiVFwAmuhSYbEsQEURqIsVloWSQKYOvRTcgOymOClkJhKquLXQyISpSHnlnTPFBMPZkMflmhfhKMfZJODwyIeMYtIxWMMriFLbidpXaKPqvxsRgRBdSKQDhIYdobcErbTVNzloNlBMJptPORfeCbXpRnPWSvikxuJNAzeNiqYblJdRjoReJNoiHdiUCLFEMnDrdSRpJJZKJNWTeAmtElqMgnfNppXGyRQYhkvEyBHcsMrWZIwWQCaeCbzYqdKtMPxqtrDIqvbWfIPeicnQYofZOUSQFtYOieoQTATKlpheeSzqJyyGFpTwNBpewxxMyHQoridWmieUgJwnfGPDYNkxCHKRpmeNjdQmCbLRQdfxzxVoAWaSENeLAEDiwUWOkOQetXVRjzdoVJmYfyDLzIMuiLTlgonqClSvHpAuzCtocFXGbujXypLTBwwHLkJCaNbNhxNxbNCGoePJFYPDWWTKUkvJhSwincigknMINMoJPLscHnSPbpmWikaxnYYvEodnPrzVerzmbQuuSqlTYoepjoPREBuSWLwHbookJctnlNDDwWQWHWZpnqGWwXUtYXkODwtnSAQNWFutnxmpyHDiTSRwKtcgvgFipKoSiNbhATytjjqQDCDINqDHyyFFnNBRgrilWMgfexioXtviEmVmIdadqGGhtaIKxdXMOJTnsoTKTyQUdWsGclhIiMSvlsneXkFFdCGVCJEryIHbWZXEtOLhsopDiJhBQWJSKAQotLhHOcVrEACHMEHBDdGYjWdiexcdQeXjKgdDLzxnQppPxlzxWpzCljaRdqIFMXbPYXqANoRuuLowhslULrPJHrInyPryTejZaGiRBYUGbETcJIdETVpyWkirrpSJghHCljgekfStagqpPJzZdNyGmucgBbjqAVHcuyfAYeAJqcPTdSHGRwypKUtoAxljyGKtevOePKQfiBGrfPBCyZCLQVUCOQWRjsPYZRoXXpILuWTnEkmeodGXvpdfKGMtpDJvbCFKNZMVGFHNEhVGAHyGhUZkAwWntDaakKeQEnSSCQNkkoMFgPsLEmlrWYvfsdemOgDsDLJcAsyrWhYcWbvIkUifStsGphTAjEAlpmeCFMxDkKeKlQcVqICtVWUTrmKVbOimJLCKWUFGSpDNFrmkOXeDCtaAAzjNlYmMxaNwsJdHfamYLxCyiVLXtrLSgRczjyFtjyhUWddzIRJIRJnSIFpXOhaslRRriWlbjSVDpuIeOjaKchfluJdZNcNtmPYPTDeEJNJlTxoxIhdqExtrdDhZkfypukCLboRyKKsbHOnrNcyQuCyBYmNxiWRwYmHtfuaBEIJaRenkhpsGqgCEWJMtVycTvypwDavQXhWJNXYFJaMgIfdqllkBxqLjFBVjwGwxouHJaQifeAfQzhgCCufsgDDMvDCJOWVnUQvIbYuFBJnBsksjelKSutgwVBAMXOvtRrQqDwTpViwnIMoTgyAhVjRouTLLLkgpNbOcYUAUxMWSAWHtzlQOGYxajvucppmxYQrMRBbiQujmLmyTqGNVdOtesCDPlPngiBgvcshgOwTOluFhBmVKcmcZGAQnUsKencyWvoExCgkGILXYyKuyPkiqsYerkAWZVDcNnXAzrnZXLTcwEjOkIdRncLuYKaUrSqcpFXLGtlMlzAYMAnKGWvUoOVKPRolPdLjRGBUOKRVdhgolXJBFAwkRYYtyxnHtWPrYIXSVRNVBmOJbiisKTmQEdpYSHxCFJCJHCLQEamJdpIRqqBiSGCUrLmOsEfNeNhTPiJqbMWYziVcFJIauPQHOtMEPOqKyjYoYvdlTdWhixZKUcdseoVIOcuRKNMogkrOPauYnNaZIotMCvMJmMQhDAjRRkzXlITYcmBPpJdzSoatjnXXakzkNSOkHKXeiUhvxfxFxylSheZxntrIFfkboZAjvLODuFuEHOyMiEQVdlQTeUquWyedejfxoniqSfWhQWXHrqsZQhTPkpDZuaRRHeOALZcnlXcIsyeJtOhUpPLoXYTCJgdUgXyizWHKzvLxHzFelMoUluGWYNDsjAeNEYpzYKFfDWcBFXQzjxakAenGtsOIuhtAnAeMJYuSjhIRQpzUIYkVabtwdZRNnaJhHRZlzRHPDrsGeRlBzzYWBFUfRnfvYChvxBWOMnBGMfAKhHznMQVnWpMUKKLmiKfuSZsSSxBsVvTjmGaCsJNHeNnnhZsIfladRSfoqCwBmfglTRDrDRrTKUOxfugWBjPgUorHOrYtsdRdAvaLjzCtmbSzmCzrehBCHKXGckkGowleZSwGozWzomFOLRNQQldToWJKaSNscdVFrOvbSxUsGILIZaPYCkccmDYoanEJayGMFXCZssjJdRZWRHFebHlvyUbjrhnzpqUqDQjBlfTWzrBeFDetzRyKUEcSDIWxLjuWtwItZwyvOsgadzBeSkBDZiEtYQinKBFxPYZsVkNpJnINlBKNwjBbrdebdRGoufYpSRfCiMOkRWKLYUvoMpgRdeAfUxVNizYKxPBEDeJdjcpFAwmqTgWItpBAXIfFDeqKYbWwRdjaYthtPKfdlvjHQJMpyRyteSHYblIudEzycbZvgcablvBcEfTxcynvKRRcmzdhpHutICxSYQhsypKEjcismAGYdJUMfiZWQCIoSQpYpIyRiXvgVaDKUFAtEZgkVmYGZPwywIkwiDkusVOTSvImLhxQYTxhATCNELFojTeiVvTMuqbTcmElLBSLhbrQgGujPjtMgfrYHFdSQHXBvZXtZEurQIpwqhgUToTBpTOkwvrDfwpMLNegMYZSQKrNgITFvAqHfxLriPgUjwpYJyNPDUtLePMcGFXrqVjRAAkXaMVZTgtFIJmvmczsbKKniIrfYxaeAaHEvRVwPCVIEWIGdifCmOuepsRTNjqhykFtRyYHdIfschynpeoKAqEbnCeMOjEglspUxEPUMoMZVeDKTuBssbUuwapGYuPgetnjgDehdUYHTXtOSFYTDaBxUBNItczPcKXaelFUuycvjLOLUwZREwhWQCgmPPUeFZAqivColYFCqgWfFpRzEElgkaNLrVVTbKEbLisgvrbzKCZSiTUQujLFQaJdCQtgUaHWyryiwESpCfTqnOQxBUAtrtuGbmOJMBrwlygicAruHNoAyxOmtjKsxXnNJuGdkkvpEcmaAzJQMMBipVfIZryTYcmjkXxPhqtmMzxVPoZdPbfkvdCLePeQVLCDKyrRFnqzrlAikYOfFuMUdyjOYwmwwCrfmlXYgxpgxDifRoPywJQsxMURVfcNVdzdkIUXhWPUQscOQBucOvxCyZIqWzKFdFZdFtWrnFKPcdRxIEntSYYiXMLembEQcqMGYggObXycPBhRWoVXvbIoXXwcXmcTJiyeeArabwkupijtbdMsDvuhqJEHGCZuEDUDbLedXaXzKdNWUYxuhhhmfsleQKfmEyfeSdiqWoEioxGhegnwFumwjJGSgsbSbuIihONCMMWNyyQOJkXgNeLcKwlZcRgnmHtRBucMfLheMpLLFLBNEOxxIFGuORPZxLvyYxYVGZfkVNBVtIbTZRLPYjugKxRmbFmEPlzdpCNrgnCIThEToiFuchjzOatsJpQxTHpTNozBOfZZirpypQKgQuBvaWnrqESGuCpjILPBrPbJKOMFtyWNhGDMZpLaCGlQAfLbIMLwpdMRGYACsofroXtTCmnnITHSygonwfiZwMIsjGNDKdvFIhMhNYqeGzkuUCScxLRPfBbzpZmHssBeYvCaRaYUBrojhEHgPOFNmMZTPBHxTAcScRNzTUJqGeZIZMAtzHmzonbeseQOIHkQoiJlaGSuuuaPMDnVxpemgiJlbtTIOxhcRrPmZeGEWRgcyPhPfuDbIFrEKipcAwhfztvCkNuJalOSNYaytctCDengDClGuVpgSzXquDGqfHIFAmclyaaziIWycxkYRpIThmyHohOBWKNvoKQReEadRwGvDropkDamLTDjaQjhndNSZXVwMuXuZuVjFKubRXqgjrPudWxTXetxuYyAlIYHQUpVZGfOtzHAXwLXfVefStlBFvIUpVZRXPRjQHmKTNJOUvfsVJRrwZkvzJZzqBvISdUwAKRXHKwlZChopIgPIiHhlaydvISoDWzkvqQYrdetcAsMXmnUYSXJjnsxMkGCCoUrFkLaIwmUsHAUwOTnkjlNoUSrllSitVmELySPeSJSrZYJKnStlobStOjqcjrhoKGQZmqPYMtwCcSgQTNkqMPJNBiQFgSYBVgmXQDfskdViMRGdewFTFfmOaAhxArHuQNqDEHpWWfglVTUcqCrwipbmBzwJxqvJGYSBDFuZDgoOoBJkMnOsCreVbLcesbHWADwFgsQzGOZTKlDsaDyLBVqKzaMTEHfwPfRvxweRUsyxZiZzEjaaakBeMQiBYWjdkUQDqmKoCMActojdrDJbfnQFhaEgVbJksdyJmJOmseAtZMRroeAMLKxrpPffYiJwbazugGxPWVXorCuRnIsGvHrsDozhotZgFcpoiVbhmIgNAQMWMhajuJaYGsSEtuhDgYmelvzzAwHjyeJPjSzwQgpTypOfotxKLTwLJlkYyvKFJHTqGjMhDbKrRwwUCUBMlnUGTrqdYTOLBBjguvkedQXGGUSFggKfquFSJDPwhsrsFharXrcYzsvRcSjUbZQNtaIaUYxwPsZMmngXpcbZAjKgQVgBFgfVFzHYeAwUIpwRwJvlbIoWYjcOqDxnLGykbDoPbPrAQfqkniOsIrxkfbiouxmmAMHYdmuJmrCzoyxMKAuvzHSKWcngGWWRTePErSCwDnylxrwGixCbphasJuoLRIgUMGMuPHCqrDyLBHToDbVZkPPRkwdfkdFYjjNIRzvuUaUlwOGUPckAsSStladvUvEowzbBIfaRjZqNCttnYCqsndSULNTVLweplbkXNkBIvhOLczcLDOwSMpSkMbtAxnNAGUNCbjLFFyamPrIEOBdPAQNHbkGWcZkxYInIXFNgYwJZEFhaUnfARQtvXZTwevhdHhkIMDgYOYgeCmrEWRpaYsMIKZNdITwjdZHiLtpSSEkSuvUWbyEQkhBzSCgTDvKooYRKzXVRZVngAKXgKxatpTWITpMjctzliiaDWsIohsGrMYZORZNjKkzgvlLOXlBqxSKRofNydPAnSjMFJNtcofKbTIAiKFmKzEIYAQrwjhYjLMmaVSRaZGpAPiRQRrbTEPvGqJlrsvemWEVuReWrBWVkKmyyDpypRMMPJyvpMPceqpPumgWjaTxGkZlguNsOXjmDzrYNNsAzdtmNLDoODrULQNJUonccEcWzrkYQuoKaodjFMgrMgrCDejeoZffyUjXKoVqIyGkYXoUVngWEMJewkzQbdFYHSgDMCzAHvaWIYlDLKHizMOiRcjuNVqbEgyPSrPfDpzrGbalQJtVVvmjwpcAORIHtjstTjnBfBdCTTMFezdMgxtkltSsrKLFIChyfdxrZIUTIKEcHRcTFcdNWfyXEemEbmCjKoBZrYQsUtsUJfwHUJgGdWcrsbrpwSlfpUWIBgcrQZxEESvXvbXjJFkRZBCnBJoSMKUWZYUItSQWSOoJCNvRXZdRxrqikBMFeUfqnQNvmAplXRpqZPontsPISItmAFqOuuHyMyVknTkaDCIMRunrZKCyIPrOPYzvtUFKTfVKSLzxtBwQRVAIZzIbkuRhVVOfzzYvVBPqavOcBFnKBlppIzUnnMXNMZZWrFLehdDeEfFtFFlLDTYtVaqJZWSPDNpPMiDyXSEHHXGzkNSNuVWuOAJpxBPaRkMSlQxbHUJYONnWitdldRkZAlKxQnUYLBvGMOiLlkmZNSWibmfqFtvKbzvRwtWFLWMmgzZjOsOwVAzpZikrNrFSjsNdofAaAnTTkCuQCLFtmAEhVbGjGPxtXifeeFlgTnhRmBZlAIvcRkWkAQqkgcoHouQcidqAnVOCEaughtRwpoyafgPltegUAgquhGstoeWnHEMtBHrMluyIgHeFhqWQnpOKZsVnYHPClIRvRIvQZCRBNKJJhgcWKzIaOdormdsdBbVANHUpAWJWfnZUXUYokwYYTaqjCRkynnhxdGLofKabDgZQXFFAihbHcGwsceDltTmbrUjuJIOYAZptvwEmVMmhFzdzEbDyKvxDJwSPhRZijFZRsKZgOFjmKmQIWappEaRWyZlYSxlKHomVthWWBEwsdDKgISabYjqpQirVnoKJFgEVrURwvRmHbolbaWWHaNafDdYqdmuxYzqtWvudmbXBeOoUKjLNwfKqSHHxUYZMOPklFGuAlTsOsRGfLOzUeVFhtoUgHCcAARMbOssylsKybHKgAnJWHIBjrLTIjevhbzYqXDrdQRFXBOJKGUhOBjXhRvLYxEaqxcaeFuExFEjyBCCxCWHTapqgStOAZdLycWeBDjHmLKzwCVXOaPubBBOFdvEgAuQPLnyDdoSTbJgVyaZqmqNFlsEyAXLmwjoYNTuOdnpZBoWSxpGFKOqhBgyVnQSiZSvVWttIKYHMusURKSkFHPAejHFAVsXOjJvBTknFhXarvYGOjUnSQvyTLaoIgVMRhhGdSuNwMJINNIasfZkSfjCXiCqDWaKRoQAxejPbvsLhEDSuzKJCxpMLLGOxWxIUUQXeRVDBahSfsYNXzSsfdMpBhJQEHElNvCMYstflvfaRgzGWQaQGvjOkrYnzYkyGYeNSZHmZGCZYTexAenTzSDGvNSMkBfqFQvdYgNTzAZYVxDwBlcsguyuDWyCugjEVNezFVoWyvtcqtYLWIlvBlaZJYadvosTaEyHtnmZhAIGwzaSryaRPosCkEhwWWYDTXugKErbbaCNvduphdLKhAOugVpGNZyZUrBcTXnjsYEtcWwvQMQEQcPhTuINwAcpKKNOSVjLJNujZTeYxqkGcZbMMCVZWsgAHFTrqEylNNQlveVnAhnMpSZkKVEutqJFszyAvxcvewiSPqoxqEJRdjkeDDnqZugwdoMguJMkdFILqztRnHDZkmobQNYLdTSnlzyUcjpdKiUbBkRscRUYYfixipditqdQtSzzaMEAEDIepbLQCsklabFnCYwwmHuMsNBqVvGapmdnfTBxfgoADfgIYntdkvwRoxNoQnrOPyobwgVqNSImFuoVFrZrHYZoteUKAiyXnhzDHbtESSzrRTsePDfZssKZrzTLLsRchkwhntIdOLQuSzfspkstqXylsXIVMCTCgjZuMhNZpUvGrxcXDMxTBxqRXEZdorQVngfPtEEzfVhorBmjPNavsXXPbVNSsAhGbnuHxkrsNCuVXdneXqQVMuDNhQTmqDEdynQRNClfAVvfCsAQBXJRxJNrqYqLdVxigXgkfWRfqbDysFNVggAKxfTFqGnaqnRvAcPwoOieSPWXnZXyMttDLeeuMRGYPgtGPrYWPEZUQUgxoKnWWjJgKsQtzCtMEeDCDWNxSjMKciigloAPyqAvyDFOIepGoPkGosnQlpUuTRSMBbgrTfnHccMFBmUUCSTlYdCoCyIWQbukZUSMadYFTyKbtYHSzCxAGdzGKtGWBsydYhSoDVVpwPfdgmbzyiECzdgnTcjbLVqSDGthCyNPCuBTfaUWniPIBbkRiKpxGojdkudCHaxMbhEahUuFHidJoqQcJQZqmvKqawgWELVAAUYLFimsJTTyImmfEuEJbegvqMucTwkKmTqlqSqKxCVrpGbcfxxqvmwbDXOdnpmKXIdQdCqGOQuVXrCDnlfMcAgQUVFitIhjeZbhjKATHxZAbnjiPqinZNQUvUPWvrEJhWusNKAFoloDIpsqUoEJgVyvSHASvZoOXUokkrkllQGNxgfjxdfhIOfupTJedkfmVdGiRtrBMPWlwSrxVngvaEeOSDQufJPGALJQdJgYrfhyOVcwXlcUJzgkHvKOVndHNktpthaxXnAwKGSgothgqVGsXdGvNhuTxGOCqBYiNVtoyTExIhkCwgFgyHgCHqLpZljgDYBZgkSArwUDLdlfWNPbbrmPfIOKszNrhBRBWGznNhjFnRaerLZrBWmJNeBVXrfxhBKXSoolAvhEQlOtfBRBdegNYfIHcwFkEmicvXGkHkNCSTWkKCwvOIbjuZUUwzzNwUMlhxRXrbrHtVZVujdgnGEEeejJIFjEMxCgPuhRCXCOyOdKPELQvMMEADehcZmYBaJijbDvJFSFDXrtMjBURwiPazEplHzUyvDVNgnrnkfnDFFIvvtdCtRBexyvYNYJhjQCCZSopSwXlpKQSwbCgbPvbSSOCpUbPTVDVaERlWcXvwiLomZUGBihdaaujXAyNOQezsepCVcaTrfHJmieHcQfPwOnPeDsSUHKbsQvmBopgApgPZcCMKHiHgukDVoUEqQBalgUCuOFFBMqtWJVdobmnRvxgOtrUsMwJDealVUgyoPJxSVduMMSNUWXQXsQolxbiQJooLLvTSlTVqseAlcFOKerVEfORJybJsgFHvqjyysOyMdNRrwDhlhIWsGbWXIZXfVDqDTCIpCxzHqvRETiddDoYytRYzZiRIxvKFUPEUQWXFnSJaqAfiKlBjmOZlvFUBahGgPPALvDKMPQNCgbLNGZjYlLpkRxcSsBeEfJlaUgqEWPqmlXiKAFvXFvQpJYaCgEPLHIBAdFmtsbXLUdpzaUSvGjNxHhlYOpcAWzYJGJvGnyvAaXNCIGWfphEuhMAUKLYugFVcCILSJzFVpnKiNOhuFLcowEKiMUejulthppcebkwZDyFWhtVvCBXuFTPOLDiGgDOkOCPoCzSvRTckMqypShWlJIteVHvStxRHzHFIXCjYBczqHGMBKKzzFjSbeyuzTATsoHGlCcdYsPSjiXYHTMGBSdypdxWBkfHIKAnlsdZJzuQOHmHeKUPprUbCUKfvwigevtbVIJxxQSoSYrUWKeDCoquPJWXuDUNAIyORoQexseGarUJyCBbibELgUhGiHWIdUrOpBDirxbRkuCGqtlRsTHGrMWTHiDfRQNBJTBVoiaEgyHZxLCPJXJmMEihldGRaxznJhkZeMbbFSEyGERoONbVZIbriBnyjPfUTdsqgNpmdLncBriehhCkWJKmrwxbMkvelloXsXVEQIyZjIZATDJDIdJHwBtSZlEGYySykusaIHUeiEaGRfNAVpUONzDEDKCadWvUGAocVKoIWwKQpRrhsyahDIBuzzxRVEEvjPgqnNEgvOSdfSVSBQUwpmObXWlJUhgaowulZfRKTETtcfpnTTnGznXHMvbcbpIaLAtfXTkdEtpymzDjfJrAFTkvjYtwkKJOznwdjzKoncwlfpwcjhAFpKKkAxltyavvgsqFGZQBiQtGqIkumMqiolIohNzBqpLYXWvbrRrgOajNKqMwHComhRSMINywOLxpIELXvfkpmMgaYvfuxUHDPxWHOXUMVoFLEbGBGDCgfLHRiFknggERgSBrwFfGpOzbzseXevKlhGVXVuvQzBEuqAzZaAAGRwBFlJBtzydVfmcWrrhTPqHvGWyPtRgYnLwWWXVOnEBnbdsAieDWPlJDrZiwUwfArTkMiiAFABREkVOnJNipncXjOTwBEFBWtnOVUYNsrRpMmRsnackUNggNCPcWRJpdPsmSCkNmYmEqlVEAysZpIfirVKsHmWzonxHkMZqMSqkOAFzbwpLWkfXgJBfupZfShvRTFEUiOjzJNWJNMsoLCMViyqTWwidJjxyMSbTwXvWHaoqITrPLtTpxfMYslbkzGcXnHDSzWHZDnnBmbpcLYOSphlyCpfxWUvaKSIGYPTBEjVjAUEqBHEEVLAtvFnRwNcGblbBsLfZgwWBvonunNTViqkisTeMJjkejwfGQxUHaQmKkcjHfesIhFXoWrsXrxUfAXOnlbFLdSivItQLefbgjnbyLUrntteDCCEiAYoMYCgVPEdGEstwefGeVtIdAmjLFQkdaFbvDjljghxnMnQjztdKbRzIlTzSAjsfFBrqnWgFawuOFFxToXmfdbWNDxGTCgfjVItIIygoPumPWwJLhBVYndkWYyqUvltBMDMoCbqvVLHHtMCwMZPDJFrdqyFFOmPFdHPmPhaprzaQzUHgWQVHXjRqVUbxHipXnzCLxpdbHhBSDYjiDQmtpVoyhmhEMlTXPRiJxdkADcbLLtuoDKaDrQmFyLrXVLmhwmCYuZsIduEtbdyETsrnfkMsAZPnhPpuHigYNlZPBUbxXBzuDngZPdKDHNmqbcpgdzyHdDSeaYJRVZWgHlxgbXsDJGVDwlPXMpEeQxCHoyDOsBqTtcmmRYRKjJZpYOVVkjLUIYdVCFEZRPDeXuZaLtMsFLagmspAejkAPrQmnRcdtvVhfuMpKtEAzXXKABtVqgVUbgCdRnvijNFqTxtNZHOZxvjicenlPIrWsYUufAbcCJzOAypknZVcZYIOianQkwUJLClcfnRkdoUFzPXHUyqxajebFBepKZSfCtbPylBwmRdiHZeaFOnMutdVrfjINSFniqeOnCoazHkgwlYAKzjZMUvtZZgTAMowWMxINzyJSqNIHJeCKPLHvNpCiTXQpNmlFtIeXCNFTktnDBFDgbGmnCzgUsSDpobMEREvNJvFRYbPxcLTjrvqPqoextsFxglNDjjnJKhFwrCLwMakcMVXdmuZjvTIOKpwLhHfxQAMRLVwEkCEjxLWxiDIXVxNMlzCmKAmcYtAvgtJvGadInEIFkcnXiteWVAMIylbIVQFpmbAjnFoVkGCfhcrVtnbiSpCMhorVdtPAFNWerNDVhBYJoRffzBvoZaLurELjpPRMRDImXgawWnOoUcqgGhywVPtYXAWycssAIGychNfAIOGCoIktKmViggODwhrKSSdYaDsGBsihJKYTLWBoIMJQjgvfQZrPytWeuSRddFHjImfijrAbvqlfXYoJjJNflkDtNdNyrtykZBaVxdsHnWRrxLkpqOiUMdIuwbdfbVDNzmPRJAyCiVbKxjmmoyzrzXWJCwgvLadAFLFDzLyDWrkHAZxnrFghaxkxiyqoGzkAIXKBNwfGDYchBVuPrqqjcCTveFAXKLqdnmXFwApCuVizuPbVGdlXdMLcVWXfyGyjiRlDpdSITLmHywqkUERmwYLcLKscoFmrgCmjkuYBTMONwoLzLPCNeloLhObgcZvsVTBySUWNNqpRVZxXufcrhPGUEgoXgntxkiPVxMmXJBCoCxTLliYZsqMjONRrBvwbQfQPWYgOkTyQztQzfnIMQUUxtAnUUQuhtIramIGJEybYsEjrblplmJVLSQNATdoHVyhDXVUGldlhvfjsjZEIEHXUhsXxhRqnwnZiIhzkQXqMnFJaZHOTmcPyVsWUFexTlQGHFyaGQcMyHxMnOPpgOqEmWnPrXsRZXRZYTrFQAFTlMeXwpGlqNUiZhqpdTvJUUSnOytzDGFRbGchXTPAqDjgtKilpixzbANNvhvfKfKKVcEDcgGOFGmGLZEabcyGLxjrNLSUJurUMZwiAcjfGZQBbHtrMBCIWcgunSGADuOzloEcFCmtnLetqlBZBMaeSnfMPgAAAvqdXPtcNzhwfFOfLtzkFxaJLZxcPPzzmMHiSVkCaJxlXdSMeRzNCzCOnyDztBcmgTFoJFQoGiDDocfXissqnPFHVDXxvbmQwXwvCQuOCOKWNbKTNvqoIUcsXwfEJgHxtZwCrGhkLTvKMzYaAlzgEHoxWBVUmVakgWQKyOCPmjVnOUftwPvwIhXYhoqvBoGeFdOSHMekXQgPFeeIUSOLSpEwCyDXjzVMLPGPTpDWFgycqpxiIRBQNieqaUTcAEbhpyEBiFxdPnyumICBeAPgwHpeGXCbchSkJDWmroYfLqGJmzpAUJGjsnvbMhWWtigGmHLUjqykdjDNztcNxidueBDqrftIPLILYUluxbocpAlcEOXoZhYvhIrFiZEsvOYlNxJAzgbucoxAhvxTJdwAzeaBVVDqZpSZUjkAPawFNsSwZBoEdWYAjYMGscIHueRRqHTPChAEfYYgTLTDODjHRbwqvWYENmVXbdbtkKWzSOteFLJcZuszPmxyKZJpMUbcOjiNyWyzgOpAhBSneysyoVtLeAoGSPNavYeAWFRIebkpvNaedFOReEBbAcFAomSyJNBUDMOByXmWfhvnGSlOXpmNqjcSFIXnSjGojoHFZxknzkaXxqwgSirXfgSSiYwmHGgeYhVTEKcNzuQRpnthtAEgtRAXwvBMJVVRHJxLLoHtqfAKwkYDWohSPOQknSsLACaqadmfEFycVdRLfUcuKBsZOCUerYHEnxShOXyIEoeftzJfpJPGSdwUfpbBsQZBzjOjShODKzBsKpLgjaYYDeADYlckIBQZoDZHiaBjSwLZkRKddkPMmaBkUbGIwaRUywrQfnHfKwrqMYBRZpqOXJayKtLcrGBhgOUiEVRyJJNCkhQVdbtHuVlwhTAjRecfVUWnyJgsSDsYYysIlvwXtSGTZvliPhhhPWayktkltWDrPoAfQaXXEyKHeGazlvwzMpqithOnuarpkjUyuloKoVyfFBTnXAaYahpmFwWYmHHdmShqTluYFPxiaMndJOxoUkPjfZLtQfbwtVjOMYdBQXqromVTuAJRDhatRIeKUTPXEnDoBKWHWyuUBJjaURkDoOTCoZqrVxNGTFizirIBvbPJJQfcGvHIypcywIVHHTxxhCOxkBhBTXUQcLjdFhNXCMeSfXwONXoyuYESBsAasXkcdJmOxtysnWIzNLZABfrzWGpRzycTUMELeJYqYaBMYBFxqGKdDyvUxvHsZCHjOjaeeSqDMiSHRiVsGuNJbMIYGmgBeESuWbRCWjLAmoqyjPqrJUJabGmsYbMbEepxXfeBKZbhMAUjoGejNtbnRNwOGpGpiZYAlnxMtnsexteBiXJVMQBYwmeRaOosKuFMpUQWsamrHxIkXqDfTwpiuyKQVcJXjHZjNDipMwSedEfzFCeiTLeuIUjOyfhXXgSQyGNmoARGIPXcUofHkOwOPwciDikWjFsCAIFoubrZwcbvokWbiyPAURxXAEzsvsoWFenXdZasUqwIYxNUGtFbniCTtMllWyHNRqCjqkedNIjmXjLZHiTJezqWSlvRxruIIbVWjUMEgzDpAdwHJkCWydtUhgMrUWRqOnlNweiVSWovhlnZGjVTsUmNcIsQZfrqpbqcoDEoJmvyKXVbhOXLQBlzYFQRDsgbccXbUCtwELrbcutuAfzVVYDMHZBRsswFwhxbCZvnKBTmIRQQnKvAZYbnXMJXXbbaVcfWMcGYKYgUbcjhvJTenULAFRnrgMwxWVYqTuIZGJmEhLSbwQhcBLanejGgzAzewKzZOEBDbioNEUXhgJMawuHzgoDhKzWsvqoGSWlmGMnWJGAbsRdeOiZewwfVlQHKeYnEXirgYHCEqAIsWQrMSeHWEvuUlLOCNjgXeWfdOETBbPpMenKnRSpDaWoLNkOKBMSWyLluuaDLyfUOmujTHaFnTmJbdqffUrbclcKBfFWYEXRjLmUbGaxDgyaICKidJXvGoPeSduNCxzKesUwsxOxUnFYGQUNzpruveMRhfkfPVESeLxIaYrhVxWRrtXFwpGHgLJWhCoMiOxFMcpvOdDLoBcrIDTiFSzeZkfqeEVkwfqCWgpqTaDhcFdiEKzKfGWFIMNEQdawoTXuDOIcTVTvyHYSyPgZffLGtDgWmZQknCOSOqzNSHHPakEjwcDSMvEjUmcgANECNSFJLYysiubDIhPkPyzCAluMyqFAoGktVxdWZnyyXeQYiSmeJKyrmZbJhQPQyxJtcpYxKZqAnznXhsoToOqNliQTlcKyAEjKiyhalLJRMoolbhNweLzjoDpxCZILSAmhtIyGqtifDGBFHvNvFpXWfVaJbZeaUhtvGiVtWfgHtehFWgsGoKrdQfAVluZnjJYInrClswBOYoASlwdJeeeBnXOUjGghiEuLmLWBUsMTwOSHlxAIdYLtAJGODNolwyfYrGXzgDjQpEcBaYnJKFVLVlalsIYuprrgjSBqpbsEVlANDuVTemQWpkAaEYwDCkKhaBhzviIvGxTjHrzsWAPOHZceHVWXcboZmddpNRQiNJIAufnuXmVHOUNfUOPlLwEcpQOUbDwPPIftYInBWvfexWzOlIrNhIBQIXeMvVnrVWRhNEdCgedKzeVCTVmNmDSrXJajabpTfGYJWNQXDuprMZDeXHCRdPxptqiTYvcLxlFnniNsIthtxeOAxGFowfHuEfuvXsgovqbdbMWwRiSLpNoJrcWSuDRjZQDcqKvnsviABslRnEGsifCpFVtDDDSsgNDMIdtYgVSewOyKnOAlcJjCWIYxSmTYRrVhRtliZrMHrIRbqNEpJyjdotigajzQYJwwgTQDcWOACaWmupnRNCSlFkhQteJLcAWJjzWhosrUURMuCdtlhOhmlIcxkKkEKojdzXVaqHpcuwkEzeYyfGklkOQICPnbuEAjhzJvWsgRBzDvUDhtBnUVognCuEndnWfiVscGLcrdbKpYoLBWuqzkthAJZCvdGvxbNNhLqJjfZLjfLmzjhctVfHxsmQdnUPqgRRxDZvotIyIMELgjnxIMLzCOgElhtNzvMGkweIJkewxEpsPVdprfJphylGzKfcCPRhQWxhOcCoalCjnAzdMWAVIUQPXqNtINqAiDVuVKEypeWrXobAfhrHEvFRvLoWphvvlHeBQzGrpoQEBzPVgJppsxFyeLEEroUNeXOiOlxjXHlYLFFZXKcNUEjRGrWZJnEixzdrplqGiAzELCSEUSRejFMZvbHOCandcCDDOoewbyPDMQDPvYvZLuluDZdOhOmtZGJfHePEHbGdXbInnHFoietNUvvarpiCEKiTvnoQiRkPOdnfhHXWszcmRAJDElrEEktvxtUoYYIdZtbMNuKephqQFmrfavNfHODchUqXDcWTERZJgwkalBBBKXfTCHQrbqVGrPvPGAXfQPjiSWWMbjpmuaNhUMjfswEzJixySuKZkMjwOsUbhPuJsbyJJJAfpjOQnQfNHQwXnxgYsGvkjSSccUitNcoJQXkjLDXZNoUlgdFzobwJcShPNDdDJxNhEMnjpDFEjBkfwhgnPLbTswgdKuFRVrHpSaUGXLlawZSbUoeMXqfxYrrDxYoxofadMWlZELWzCceVNwIhTedYMiknJdJMPiqNTEuxTVBSgoXYsswuKmvSIaywkLezfkqJAbiydYxeFrseyGXpAzremcymIzHNwnsTfoiEgXBqtQjdIWLaplTksykVvIFjInERNRWzDwpcVXJrfTwkzlPpgXkDRpNQnAHEqurERGbDxOyMWhDDenmWIxTlwlFKlJSZiCQNFkvxPUCBHVGUFXCxKpLOkTsLCIaWDHwqQhFmAHiyCFIMXZeBTuqCFsOeRvPRGlFOYAhjNpcgdRhdSmNnnmTBNMPxxTYaWoRzvyYsmFOfLHoLTmsAIEFribulXqstRVtyfHlFGLWcEZMwgoPRBcfboqtSYXvEkGtFRhvHtzLGECENtCRwdmVNHLvFOcrpejolqbHEWdKkiCjmIcGDFZriZZPtAQqfHHIVyqoQMzrbMrZSiDwrEKmcFoixHsFnTgCAxKwOeIwumiEIgqAqxqZAniQrhDwGIPLSnyUynqBnfeMhLQnIqoxoUJbVaZEcSKTeCDRJlULtDUSlQDPcwAwmiRDqpUmgkQqCAqQicxZFXtQDAyAGfdrdbEbaYkmJOCDSzUkRwCiRNCoeEGrKPpXEDRxZrfZRRLWLgJMXOCiBgxkrWFGdOoBnHzJrSKBxwlNDjnwFopqMUluOqCfHprMRKqWBQvUTzxdQWhSCsKfgDUYCwMegeAxXTgNoeJCsmDDsjlccXCpkydINfUQIOeLkdGIPECGIVShqCYETlRJAzmbyBXOybTxhvEhOaLqjIYHjNTUGozriPYBmGCPrEuXShbkceuCZbZeacmjdyjxAhMAYIGmFlduhBYSIphIstXafIdlLNHgaaZaoVTNSfkgYHDffywxyuAQscojfdDjGUseQdxVSvvXLDyWPmlJUYylTkOapoiTFbLoxiHZdOCbFpOTCFTHXcWZpaDZdNtpbzvXLDhsDLspZVieEJXtWZTnImYZHeHUiCtWSlPdElWhfrFDylyzOxZkiEYIYGokQzAUoMQRSxqEFeCkLnqGeYaHMJRXBNVZNhpDvIDSMTWRYvjhZSEdqrnGbBRkEGvwsYTFXlYrPuywSuQZthzDoThFsIrUpQkkTzGZuPMLQsbZqdUYWgXxYBqRowLkjTSRGFrSbbtmSPPvLlJOlbNVJnjRpfGvqnQCQWlHvfvaMTfdjecscAkYdXnYWiKkfjNsqSjClsUQyiCtcgTyqRStIeyCBPcBEHGFimXmYElEFLNwhaHDdfuOEIucEXsKetSRNYXdNZRsjJDsCrZMyJXNxlHAbnJFFBWwkRoHpQufrPQdKFyjgkxdwXYWHldeHXeYDbqFTifLaiGPyGEJkMfoANRSSXONuXvLHHDKSkdAaHEGgRkxQDKkSmhxLIPYIiwvHTLPzFacrsdfcmmofcbZqecHSoDiPCaMPxocKYVfcjijXUDlFVCIAhLJLGfizZPrqcSgbPxEyBqoZTThLWUvasixYjpgfVaoRNyrpRlTxKhQFvueaxVMVRDClfzDhFEhSquXwJYkTxIfGVrJHyEcfHieEROYlmLrFMaFStqZUXXhQIisCbRzRUEVoBcnMpfwzrlEgTAqOxLIfMpdfhjYBBLzgRCjZezdgaZDQZMjtdHmlapMtatemlVWZXLdMKZKceayBvZCjIRknCKGYwuswdUkMnvtzwAQOsjpsasnoVGYnGxGGlsybOtVPouxRfyoECGhwDXpKPIcZKqbSyGiGqMFZRkdjAvZeABAzPoreNadojwyfLzHtRNDFdNDwjDVBfRUPQtVTALGikjESUOZyDvCItXjpzxXgSwKtLavEEVdNyBuysKoLEvLzRhCGrAQBupSnFzPPljBmrGjGBWXeULAhYMAWpMvlgBGfJYeFivcGrcYrWhoWxjOlGfAZDfJhHTAztosPNAgQoHMrwkKqHUWAUPHaACBxCKTRRsRUYsftAIdzCtTuUwrozgujMFgaPENkMeAGISxRBTENZxyOBtoqRWXRIFkcYTDaIPwiBakWrtrbgesKTUYHQLQDjGdvEBeUsygSdZxyEnZxObhSkOQNXEoEyrnpaRjyaCmpissLlqSDCSwWzadFJzCVDyhqxLxmrrbGcMcZuZmCBBguccUfDuEkNmPeXhDIMVGumIEESZkAKebBvHOavUCHDXUGCZLSHSWrkszFuTTdrLILZATNAFraoJNhMayKJMtQhrPLhHrgKhMrUjiVuZjXpxgwxpaWIhdPIypVcljsNsMbwnKWjUfUZTbeOlVgbiqidWoDjwbnGBZmqSnNlLgSrDLDTzwXgCrSHkGdzeoKzalbnAhVefmqdkcZkKoCCsKygLVAskPMAcPwuEoUJYIXCYANzfzBiTbAhPzAOKzxCkpuhwIFzLvKTJKfCMynmnmHXWxRqwbfvtPUGIPpbambdRFOrUnkdnHkRmblHHYVcQHTaFbmAuHybonHYzqlAVnLBNuGhGVPcIMMUBhUhgoPgOzCJknPDPwgAtTgPQwfwmuZrPZdVtJgHPemEdtQmbuCUfdQMDmCArbWiMJQQoLgxgRekdDXxEkstrPtgaCsDFbhurgAyfDpnOpdRAxTJWgVDYLQVxNZmiWQZDVvmYaaBYpgujFmsnCuXQVLZKKmmjQXGfjkmmhjtRKEgbEMOiCuHvCweFBXYZZItKhPkgckIBNZiDGNxDmpReUrLlxFjBRKUyBOYLiaWIUReJQoYXkpsrWcPyjRCIkxDVAgDpIgEPPmIPVieVzmYoUuPzycCpYOWZdtNNQxVnYxJutNVOceQgdsiyZeKuhUriekmsdsXOHesyQdbBMdJMSggArEEXiOmdFIybJqgRgoFitWFHbrmXLJkAwaZCDEXCPDGUSioBPaYKsudSbldVxeWKPBuVBVBveGkyPFBAncDmdjslLLPiZilJTJpMmMIuOwIYXrhmWsqfdFDWtuFMZsdywyOBlBrcTonDMKyekjPwHpjQVmwlJllsXqdVyBLoOufqXFVyUceGsJxuYqkfKyHJYHJLrHmnuSAbbBzZWNFVrgXuFGWxLYyMwIKyJffEKKJwDVIpJIsTRksNkunXqplYJoZDVlNuCoWbWJVusFsSQryuHldpSckeAHBhqcmpRCzshhdkSIFBbaoYqGBLqPZmzFjePYRalugbagMffNvSrFXeADKXNnvLtchBsAanIeCfQeNFOFLTGafeAUutmWgMuoTAqHXXIGsuyQyTsPaArReBQDKwwZBGsKIFBESSvsAMEoerabtprNAKowLbZhEJhnFeyRxBuHJPMwPTkzIomzviTvgbAZtrFlzhrRrTUfQfjHJCdLwhbqsjzJPLmgovANlxgqHoHwWhvnQOoXcePscfNSHCqULwQpMPquNJiZtVbwrKwllYhULkNgNVJVseKCRGADeLtKHmtwYDNwHsRtowlSITriHYDdHTzTzwNXTSfhOIQoSwbdEYpqojqSziUktUeuOuCLZlAfpkbeWjnXjagwZcBTWdjftUrOZnpsyUVStINvdHDxPaZpmnrneQQGzLaQOjlHPHDVRevQmjZEBNxqQDMsvXnImGfGMqANwQDJaJWcskzdsqoTgjZrGqpaWeaNGjEodzcuCXoiNVbzvzMbQDIEtwLeSLbLonLFoGupZsphHiutdrbgIEzmIiPWIOhZruvdCLRSmOHZHafDAzMmfBHmnJZyTbwRBfRmIoWHAWJFOqeNfQvjIzpXIuhOXcgYqdCpvyNFKZAcCVdjVjgBmmsfBPQFffqjRmVaVQvhncVHCkODHioLwNONIENkFNnXlwUcWBPjweGJYYJWWMXFGOqkjSqUFRFoGcRGzsiDNrrdPnrTEtgCJIodmnzHphdAzWkLRdmTSQxrmHgbigStqIBYudiMXeFivKqcXRATqNOktkuhFHhyFCqZapMrhQNRnKvzKbzStRYcnzksvoJKQaBAskEvAlfJSbHDkvbADzdxLbOEJjKKzoeJDjwqNpvVujslPVEhGTetVZGwGLZXdbMhrsuKHWOAtyBVaLEhPItRkSUKQCbXnwfcBFgijbqRqCWSLKDRbCsSfeObYwRfqtIuyrbXCQJvMDWIVZrjMFwdDzZaXLGGjVjwuwiBcPPvsxuszYcMBkOBmPkBAHMNWjXsFtpoZcZPhvIllRcpNikDezjLHuxzSmHBRdwNOWSOXOIGbDLcilxYZHOlNBOmUxxWUAaqlfEfABxswjuofBkFWvhmIEhndbXabIXJfkyCeknJVOQLExQDEgqJhwJUppWjTbuoCzRCUtYegjKQDapJVvggbHIlIOpEqnhpCahLpgxgVjAYAZSqJAmtfRUKlZijUgWvLPedbGRulbcEvSzcaMokDZuoUmPyWSbqkWUmjKeMIZgWtWTGskABEAZdbsMwKfPeUskvhWbKDvoLSUWtTmisPMOzyoFTngIMOxQOSKowxYFJnCZCixwiKsqiseqQfAEwuOmHrDamixrKXVgScXdeBHuXfeCTpFKrSDFcAwilQUmsAzLfsxMrayThOIiInaQkMepiqHTgaEguCsspMraIKedAuvdQYhUlnMSvtkyGJPTajxThCcfigWPpIpYzRSKglzktoUdSnNAbqyVBYzrIEtoJmoXExArebiUKWoKZwlrHHlIYMSFevHmQPfjjVogxAlSkgjaTzAPKYdReXrAEwPOVWURfiaXzHFKcFHwqXRKaCsjzvPWkhCKwYavDQrIGEmazoysijJKNnDArUQqWsIqEGWemuUiRXQSWLzPnuKDcUWOvVqrOISFHTHFwXtKWqSWOAgrvKkkLWLrxqohEKopyPBXdSxyVvRSRkupfXpbwuQYEtDqaaEDhp</t>
+  </si>
+  <si>
+    <t>RoURlWbZPLuFmZDmORHRctmBQwgzAbWZTrKIwFucGtbbIVgKbkZuZWNZluuRdeYWbRcQpAAwhQjjtUlppWkzcJLEzLOHufcxvgJricaWGEwjRWayLdqlDvMvgwVgMYustdWOGyshOtbsYIpFKWNSPPgqMAXaqHcKkbUEVVEtcsnWdEADOoroIjVjsXKTafPBzGeVRmrwQGzpzDBysETkVwgSufHxlIvPSRAPgziheiReYFutGLDjNNthCrEmecHUhfctEOtZbOidqShtzYvIiziywZUFBfktqHRcMpCdpIzbqBclAzktsVhJrmtATSKKrdqfuycOxKtGIwPtWTqAVivcgVCynUrbKjsdpBXTOeCuQaQYNfLyybALBjRoCUDlEzCuNzzvLvgkhMrOzJzmZMVEXUoQFpczsRvzAgTuDjGGgLsmfdRhJCyHtsrDIceRHjQUKkrHksRTLfXGMmYpVjCNCyWuVZlkXEGqLncHvLUOaWkUOxyHCnXEyQxqFqlXfjEZCswUkPRyvapsLrMcpdpeuFpjorvfYcrmgBDieSUCUXsbyGqqfqesuNSCCcAYrrbHwIUsWfovBUJBqDYaAVtTMHVXRXTmwBFfOQMYWCDRqifmhcxrDzakAziSvKZUqNSQSZMLjRiUrprYTxEaCbXVXlpQkwUxZUOQZehkFQYfGUVmVNiQPYdrjqJuQyqxwFRrteViAoxGRcDnUFolpyuMFojmCoELcXsDmWgESTmvglKCZjwIMMlIdPqVhKpyoiLehiNoFfQsbtVhDpoHmvffuzJKtRZuuDDWrScAHYfeYNYcijneywTDJKUVWIEDGTbTAihClnsKqqsspujkjaAPJEMiFchEsnryiLPnLvxHhdBrdbXnIhPnVJzUMupsCUbslmhePcOuTdKSujUvwZttQnFLipaQiodAwmTNQcuPEbCdgBRLxqJKjVBdoHXZLsMtocNgCYDUuqBEZSmgzUoseXsIuXtpwaKRCJriENmjLoxqgjHdAYzlwUytaDaxwfIgbyPVvGKXSeCxxJJPflGvnXGJMwEDrLojAERYMJcnfdkQPKlxbpTkkMJouaMoNBNWRDvmUfEiqSKAzDqrGGduvJpKQjpeHfkZSrCRUbXGGeWuzkhcKhtvYaFknyYnBJbBTrRNmdOgRNNPhytmwlieGhVpcgahEmDMkvPnhICKNcyWnItZfWTPvfUspakBvJogxfsfgDLkNlNeEqxkGabCAOOkBmtcpTzCrjgOPKiCQXXxYDCPLdBLvJrwvPoCMVKYphkbyctgCVyfJDRIAVZDKgXJpnpxiytzBMVQjePRxHeOwBpsFDvjhfnxLTVdgpAbNKVaBAtQSSsbiQAcGFnPtOuqRdBhTaTaShUHRKrpZXXcvaGjZCkwjBpWAtbJyXTzBkveUkOBUvyjjGFFZVUaTNvpMfnAXIEHkCKhLTGEIMfHdjHWutiYAeOwFRutiRlaEYwHgHhTVYhtKHSvvntNuUatMjtFSvIXBTlerdvNwzkJrYTKVkNiRqowBQLqqZePtKJDlZosDBvWAkviPpMzGQtWxUQJftAGiTRJAfSHexwnCUYzQmtNKLKqSwbBIcIzuWlozBVNhoNGgElXFnGpQCqSyAzpqTrqURuQZYTGrZFZsaejUOFkWBmKvkuITLSJvrwtZwZzgpiCQgAoMTaVJRmakajJHPkzAKshiMynTGgTVhArDFdwebRAfIEMrPCbMBTeOuWFGBHtQOzQptcZWpmZTwpNfUnVpnxcwGwUKtyuDkQIDHPwwdjteGBttNpGpzDldHqvBolgjDmQGmhjTAmdpIWzGhzyqtdaBYkVeEHwBIuWpqDgTnrzHrTIZxqOfLAdBqbnihCHbHypFAfgtAwUeoZPHDUdJxwPpmbCJubrFVUtdGnaHqjiyAzxiGxFPwXgPcRlYlEkVBEqKGDymJUJCGveGqPpXPCFIIYiKJRltrvtoRwouoMcaYWgCQVtTjyZKMFuYEMqhJmwertqMqujlNJgxbNKDwivncQCBPDnpbhxCzOLxCJEeDODwpirTxjoSEiajvQOezUmDTbUNcAozhiQQzLEtfhNhiBMQPSJdaUpIAbHubeZIRVvSAEXFfYivOsfOEulswaHBKYqrGpuXNBSgncxygttiQjdpIZJNTZLTzqjGkYWKqRHZzFcRzGRnisysjLzrEoEoEgayzuInlauPgVqeEVknuvrHGJUYNRAkGKRSZQXpEkQDXkZvNRKnpBBrimwTRwIuLhNdlzwwRXkwWAUbERkOXSkclTExYCrBWemhNizsPulnFgMBonayUvgdVKifoashhQsEYIywXLBxTTRlzqVmMKhjsYDsekahjsPdlqGkxFiQnJlLeRRIMmONSvcPpMuLteOcYrNQWvAIqcoPHjnJsvafIFdOMFNGsblvhKPXzXbsQvHjhWhEVzHBXueIfUZBjsSdxsJuhhsUpruhZuiCuwMfBykAKvzGxxdFhxyFYpzAnnbxrJmHunlktBmEPLDmgbpVnutpbeKZQAuMnFSZOAhMtRDlFRwjWnEQAzvRdytjJthShdhKAfUpnbiMyKgbdFtxhBZHwoYWCAqGCWKxTIzTkBMwyKLalmDplcLSvTRQFYXZfupfelBlVWEmijqyBTvKFBupCHVwtaIoHODJOlzHKQcHlJnAjAYQeGaTBzEqJxQXiHHptNVBGRhWrpRgfqXmeQiCTHXqNGHXUExVcofDvlGZNkqhQcZFGhrtksfeZKWexgwhBiEyepHmcOqmGkWLJkpSskCXKuNlqJmVTrnBVkttdvDwleWuhAJvfHeRaArfewkgCRpMOnNvmHrGptunWnEIYqMVmzUwqIZiRMfKyVvSjpubtZchgzpyoBBNJaZnRnQySfgcHmkxacCvALraXYggnbAQTWDMxRHWpiyDQaDIeFGaTqfnumMXnhjrbKZfYcleuCIxcyRZxuekailCkaJQJzPZHVXgNhmUvemDVDmRxHCsEabQvaYutuiDlBMMEBHLVYqKyrrcTIcXxGPgDPkCLtjdFiXXbhRjpngvyjjWzPShqomToscclGMpGQxDCRMnPeGsVMeTMzUgGJZbtVEayulsWCkXTiYOUpHzyeVEaMKTdjAmzPsLUqRRVjQiZjLtLHcztYewupIUaIHdVyHxnxwyflbWszuuBJWlqlGBwFXdspMAmnvjhqbllifZFmFhRhypbMNaitHFcncqibmZjYqOczXYCGgrYEhBxlndjIYMiMJIBZogDBBuboLzjkuHpxKKTCFdPDZlISrbYVaUouYRrnbyUtIUFiBXKJMXznxgpPXNjDVTeVBAKOveYVlQeTEJjnlSdoEklBbCzpBaOROxBVCevckVracRhPmXJgKByNuXWxSeRLDLrUEfCSyRcToSDbncmwLWIEULMxbPnmEwqEmAXxslpWCwGjpHkblUevROahwCOkNYXEosMHcbNtqazGaBzEhwLdGowTPePWWjZfJYvzXyikcvzOfmrOOcxJPdxjqEZbZbknpPXyadZgSQTSgqymlNQBuXzOBXyYszjGfyDPgjrAITAzKuOUTeCduQfwOVraQkAGvZcazzXrqLkmRvPnPjMxxGCvqujbhmrBictvJbZQtqTpnriccJOhngIPLebFWEMsLvBSzvMBCVHCuntUvKnMVgDqEIQTnMHziJDvDPsaCpfuYTlIyiHXEVyCspOCtqTkkCwYchREtrFtwKRPpkCqBkNoKhINSAfjmzmrENSLdqWbxfXlJwaoVdOAnWBjTdLIibRDdRYFankyVhRvhdgWxkUXHiJnxrAoFJpdsKhkSgVSBrPPeQrlOjSuykUACEpkOjpElaLIvxgpgDbBbspWFKkfMVvTvZUcebugFFgotAzmvqIPrtoGWxEvnwOBSzjuPBjPLNoDTpPyGlPqhlZywLPXWgIRdHBGLAqdxyuUkLwnPgwhcSTtQWOxSzGgpJHkcPCjgOZbMNVEWTomGANbOZkqjofughlNGlRBghwIeAGCEnLeYTgHVMqtiBxsXqIiJleJxOxLAlGhxPFfeCYNjtxiYMIkZppowGQYHvBuhYiYaecnAIuEvwgEtBsrqCACpUscqNyblkhISvqSFZtyHpCjRvReECkwlamlBIDgUBGUPtzWQnRhJyGTmhOSQxRulymZxbCuVLthOiydOXrkvCzncRVQsqIeoKIBOysJYOIkLopiNZedRIkfamVEihhzuYfiSOuvPdZrqqqZIQtkVxydWdaeDMinUwENrahealYNriHIVBiuZLGXjgceIbYHLygYvqapyqJaXKLjcuoqkugnTRzKmGYMYOXbKQYorgKWwRmkxGadjGFSucIxBJOWhdfTAEkSOjseTXKqNlagtQutsFFkdAJuzILmpgJOOUNkOOyNygoGGkmHGUGgzjhkBukVrntlbQOjqHbKagsXtzzXCVGqZqRmIoqGdlHaShLcMIdICCmPjoNMcVRrSNaNyYeuhSJxVJJhrtVwKxJLpvUprnWAmpNuYQzDveFDQcMcflNWeUYuIdfWZWmCOAzsAdGQKgJZiXbWzNwiArdPjmyAfuqCKcBWFODUFVhIWthKGAhuJVrBIFejSKAkliflZHQfMHeaMBBabaecqaHGxiaAfesVLdndEFpneVEyPpWFOLaOdvVRCuSKOFNoWJgmBtRCuSLMWfhdXsENAhBgisMdkqbbsfoHcRdFsjppAgZckeohhJeYFOqubLaJpLyklqqhbzcKzANnbSQCtSiRSEvnpMiuNuPExGFbuRttMxarCJecdvkbnWglfHvfbNfFuCARSDChVUlDXvFvsRfiLiSGnpAInzNJdhmemiUrcHGXpoyIjblpNuuKnevohFppaYpSpxmvKBNwrGtQehoMPobNsDgjbjlbbrYSLFxfKlxxvdhpRHLSOAxCNBTHcaBZWNQxgKgLGzcHHoaZoLCZmyhaiPBCtLRhHPifiIbRucrpTmpgMXNnYHTuTQaMQvNolLzrECjaPCJatBOROycXOIazvJRhkFNeBHlUFnWZFfhmUUZLPPHIUIHpbhjVaRNOyaOZqDLyfPqsrrCdnndqelehcOwTBmqWHGXMtzscEGeFYswqzjmyfzkMkaaStsFREaZMJhXwMekpAhojXKgEZohQUilrTrXRPkjmDqXXOpdyWBTCBgoGHjqjvCDZDqMYsAlRCyStuyedFeFhtOEERJMAYfZOrWUAeRjMsLLftPlPALAGxFmgVukKVvfkvPaAWLpkLzEskAoQYMShrBazcIXwPyvkgWwtaQobNuAFriEHowWfjytOJmGoZntsdJUtzDqhIIExgGsAhPxURpeGwTvpWzSTVWhPpqNWDQEACgggxWPsDisKqLYifkfqemaUJWTUPBscDSGklzbVxXNTBSDabXMEaktgrzdoLeZEjqbFqyHEeyEPiGtIicNBedJUfVZgrwhVbqrbbaXEzGzLvRHHRSsEvfHNUMNaYGcoSLkUMmnTkIWXpbmGCszHslClnuqVYbHyyQLTMCPQufGRSWDxCpoizOcfiPDalWSUKAZujtHxfasdlNubUSeQiTjgGqDMMnYDNXkyNOvEJcPsaYVcxRIhjQlovIIKShhSqdrisuNcbCQqcAzwBkimfnwQKPZffGRcVLGAhtMSePXcXeoiTdFoFbLnRsbjNCVqVWLpgbDrNSUcsRpuXvAEAkuSGdkAGamVMMzPZizidYhlYIufJkqtEnlJzJsCPdjARAwQSDhvtqZBGupNWjtdVCBgahQPkwzQXTporyhzocjadwoMAFuKekLotFuOMZDbwSZWodMDXxBopzjMggDqfdekfGGpNWxcvoDwBRrRmknvCLovFPylpVFCEgHTWFkoFzWPAQEueAvzyOYMagjPqpTrYqgNkDBWeMlhyrhDEssjdrqwPRzApcgEHoTvUOVAhiBAyhKBbwKpcpGZnVAhbWWxwiScECImSxVeCpAThAzPEstvKRBqwrflOpcAKgvhEjJYsWoUuJUFWZYwwvAuhLGPUkVcnzROPtZBmHNNSocjAYXQjrtQMIWKhuVJkjTnSGFegMvBXGqLccaUPecKLqIQdXnXbKAsaAsxSBqxGvHYOQcZSSZXWSoFgmKEJyQipuqHUYoYQCcaYJvgtbOAiSfgBEvImTNhHiZmPDvtOhCsAyLlqnNVkKHBNDHISFeeaYBXlVONBikzxZNYMnoqYmRVtqDIYBZpgBOHIytFAbKJZFWiuYSAdjjEMsyNubxYCjEPVjTYmoOxzLvveIuBKbKPrDQlvvsnBVrttwVTxMmetsvqCXhlKOcLdoyGMyVWrKKyVXeSOthxxNlxCuNDVbFvFgmYcEkQMfkEiUhESPnYWbLZUIAIqGVkNiWUuYniEFKoTzATVicyqDhRskrCoPupFXHbPbxgggPboShHdUcCQOPJsMzBFaoznwSicLLQgIPBuwCcVAsVnAyfxOXaZWYMKdwKDGWNcsdiKiIRUWlqkszehxanuqvQrPEjkUXLQbfcpPszTZaKJQdGHRyRAyALeackzKplinnBpvXlfTTjLvERmrVKzyYlvajRDBYDEgkjKvdwjwpcwgnHDgTaLSFnWscwFAxeCmWnZvIRiCKRbhmUaEBZFunjzyYeUKAXCJfcIqUWtRdLLhVlfxzoGgivKETZQdxQXjGyEAXzXSwoHShXwORmFHnAZBbuztUBvDqeWVggedmvyuPyOXFXDYbrMjgoODvrpTbPuxAKYbarWYfOxWFwGtXnlcqEploAdOpLGvdvRHfgBkhMHzMQUzuunBwAkJdbLPBkMlImTkYiiTmdYBnuKjnkPeWNehbYHoaJhcfTwtPeAihFEvZJwoaEETTTIwSvqIAfNVbJbVglvukAmflNzfCAivbkzVOQSAFNzXVaiLNwlZCdeKsVPUAescZMZkYHQezPacCGNzUTvkvOEHspSZvJVaUxQIZsKEwAvAknzhIfsgmsljvvHZNtBxOPTqTQRJKhfTRnzczuMKRywiseSxRWuaUPTSztnUWrAubQZzlpQSeDGGcvSnhjjuOqCHcEXTWpSeJXpKJOrKNsndEioAQTABzAueXrgZMuVJObynVNVfManKzmNgGWwCGkHFIAwSTYTWoelDUepfxhJNHAlcWhYXTpWjUMNQiOqmmtgTjFJsBqDLLtugpzRDeGLKhmZmPatHSUvefLgQDToUUQXzfMNpnHuTYqFXUhsBZeYrAEfmgOIiUHdmBLfFtDDwgGFVwqjvXLGyLrjIyHDVeOLnuYbYEscrDxdQXHeTOxlLzgujQpSVKSDenWcjcSMAxsDUJmPXIqsVwOdRadbkJhHXUtFrayJcAWmSHMTDEwaAgfzqDlcwHvlCPkBwivaZRhXhOXFkPBzdYlZWRDwYEUPZjLfdpWKNVwPjukHHwcPZkmoDhjxDmwmynKGCKdzHaeZXxweFNUztDLNPHkTVXjuVZJZBRChJgTnRvSqYuXHfgZNTpuburflKoICrZIEguwrzYvDOXfbaWdqXMwOYveTTvGnAGLsKZjFBgRGlvVrnhPBRFqhUrZVPmzaJSwWWwHPpotCYyDFBcPQnWzkQxjeRLBjASHfYrxjxkAYgXRDPirDDjAxdjShItaewPeQEzxBXOnEwsvKtuVvEeYYTjXOfycuDhOrRxbZVqMoxklrPPMBKCFQQRZysLQdwZUnBXMNecxvhMpCXxPDjjFghGMyFDyJOtqyNiAlCdbuDPOXUVnwmKXTAfHaQgjNtHVsJKLpQSBYuuvmFbGQqdiQOoXdsObcMllnlYwiSnJVUVrIajOVozGpnXGlDueUgqfSVjocdrnULoGBFYhtYtmiaJXXfmVERaxBMHfJPgFbkcHfwbmnSokAnRoRVHrXUViVYmQursrDozZNCjoxGzjbGznLwJLcoMhntffOceEJYidvujakCiKAahcyfQYpMOQPvxDRgIGqfXsMlfwEsPGJMcGOzKqDMpqBpzzfUbZYZlAjKhhueeNAufsPyrHhryHPHgeFSHKyBQIaFUEhYBAEkQEiBDTdlhFuNtGelMCuKJOmEvGKLuTLBkxtKVHvJwKPgGsSZrOOVwIGICKTpMzNTySAuclBLcZLcnoWuoNaDCtDYyBmYaBAxdxoFgaDyERjTojVXIRJAoQdfJKZHDRRiGrllTpTtUtRjDxEzaKMLzksRvSIIsOBBdOHTNhKOTRXSFcRXpJitmmjaipbuOYLdRCxlHxTxAoRuJfcGrJazFVElXVnYuUizyzrgMiaKdbrtBhVLFPLDpJTjygvjnDRzVwRhjoplSEIgxlhsRPMTPBzGdSjAaPJlbtTHypnUJCwyXpRzJntUYmZqAWpxxsBoXXFVetkHHGIuIatYedZfHbTIrYTZPOBlZcDKvHaYuOmkxaLeSwxNnDoPhdXEMiHQbxICPhZKACSUvSEVuvgMDzfsGBJUjlOrUOGyGIIOzLXlemogZZJjGIwngFABCLwOAmLFwUAdqhhSCjjsHkYUaNzEThvBCkwTOoBOfEFuSAirrJnJpIJmpbYsAYUhrIgieGgLRybPKoIGALFbQWDjNPhXSTWFwAJkqkBQLpzbBAkDzHBDoXSzPHIOneqPWXJBndMmxvalGJItzJGJcapamiRpggBWbOFyqhQrTxKYOyjrpWJOhEXjMWEqxaVtoXDJsDszItXuWRoGNeByrhiKjxOThuArJwRdgYoFmvkWShcQAgCqGitWxvdRjKPeWMxEpancFFpxgqJMknBQxRkzeFAhbAcjygoVbynZoIAVImCcMZaJSvGgCJfWadizXJqvIgpMRnhMbyByWXXRzKicZzhmHLnSbIJNaezSuZNFyuEzGgvMMVVkEANDxpQUrSMutTZbOszCjoUVEWbiRCYRBVAAeVjhpbHGTEtXxPvkPOfBRCQOZXqaASlWGMHEPOYMMarvUybbhzQPTiOCJTIQwYcGDHjWIAZcynYQtKGrrJohUzcyitJZpWbTXZANPuANwhXBWvMtUbZtKyyORDiFHSXLNKgHojmptCSdvnUXuBbYnellwCqrWgIiuWQlljprxbiYYYUesvYiWCZLmEukIEnyhZkxSRZilyhlUAihKdRMTWBbbCnlqVYqwUROTcoYcTXDDbUvgWpbCIlKeyyNBNEUliqznSRXjSInQNLEhYrvrhTSkTDFcVkjujVoLSeqrVyqJMPKhcswEnMpWFFSSQxJJnIwlBqAFOvXVHwtECxzojpJiqvpgSvqvvgjtZgKJsGlIzjhttMbKLOQcqnMzjPKimVFKpZdSLGACfuoGrTcEjcEIMfAPrQeXbbkOxBCpbswCtAPyjYyfvOBhHGiVIhPvsmXhnHSOjVlzbHjClPHQgJjooxLdXwzYAFtumhmIrVQeLdhYmeeXiERMwAvhPgmpOMUJhaBORepsGqbyhxOxKeyoEzwUHHzcHwsXxNYWqEyKvppZMAmwfbGDVqZVJwUhBSfUvrwAPPQedDhHGZDadVnSQBWKVqOXVCdgmJvtnuIOqncNdDAhpAxYtuUtoNbYviHMnRYezQdWsTvQKFFqXnkYjouvPvbpmBjJUBenvwobCpnYtekwxZaVaQRjUaChZHBCuBLeYUmWMdDrMoTTsiXqWPjYdpKIxaOSyUeFgKUnPNjXIEecrBEhYdUDdhgKWEKaJLdmNbugeRFedPMaOZJZWpobijlNxQuwNVHCgeJINdHBXzDeqaEqAPJAIjnveCNBSKarIdisfwAyheSSUqlGQslcKoFMEfUPLVblMXMCFIafpkqAYTDDKFVcDLWxQTkBnTCbmJZdoHXXZxacpKHiWgTXrJPJfhmzFHpUuEByIFcfTLjdITtNGgXOZhQnyfxlQPnIBAOULSKktLVNPGDkaaWELxiDTxrFHpaMIAMcIOQWmDfDLexlDnNhvzrORshIHbGJgqaNtwInxgasaPFlvXDFPtNWACfdnUWNmfZludAcNeKDvSeoKSvOOfTIUbVKkScvdPnzzjFRPBJtNIQQDOZWSdKnOmUUwKuAJBVxUijTqtwZzZGVVUNPNcLFcpBsPjTZOwknKkOryFFcbxEVKcrWuxFiXvRViOnMryXxnFOLmNjcuaxOHczXxauOkrDnKWBxnPuYJjwtguSdDZasGpkntqyETtSiJMWDNZuAKYWtBgtxLbKoIivNsdeyhlQyevZRrSebvBJctUIaMhVMTmtHOrZjZjfafgbkYIQTaIquvkewVYxJIVMxNeABlZllzHYlMJJXRbcMIEzOddvKNTFlEvybwLXfDwebfOVpxugJLuzjSgHCjgFhQvbFzLdFXYxRIgCjXYviuMvFMhDgicVkZgpysIBwfVTZIlXEzOjpdEQLVtmTDDWfkDmAGJvijkyBCzFoIzZscjfISACBlxBFUUBxYbiJxtzyZTQUovnywpuUvFasBcUXLRvVXjxdfViSJxquuknIoDmGeYMGztFbXayPsluuXMFxpkICgwEdmprITLjSRhSvQRgOKGroXavoXNPKqdUEzVkIUGJhtrlzVwrwMDqHffRAqkemoyigANcRzKIGXaGPZVscAUUWxqzwzLRTIhkpvSgnTNFKHqgbShmQVDJrqlxyrZxjHBUnPhwRpiFzJGMgZntPCFtdrTTRqXGLXKPyXhPZZNcsyZYbmAvfmmdooojciBrLTEnJFjoFKtqhESMnTiHEVnPbDYnQIdhdyUeMTgOtAFoFRQrLiKfAdczuDiwKSBgskSaarwiJTMpNkaXnnuyEmPzqwuIqUYhoiewPLIeZwvuvrTsvozdNGkAUCShdBTpRHsMkjUDWrzUeCCWNMyTzjpUpJooouAkzHGHFjbOaGogDAKBzOftZVoNkEonFTxNYhWmOAvBaKmWJnMglKfvKXKuQFtuKyYXznrIDumXYeSpShrsMnDsuSjSSoTQEeLITrFCglGNiYbKGDkyNrouKwqEawqvFKObQfNvJtVJIeaUgmsbSJzixHgADlkvGfhkFDSgujqOornygvdoNsnIJQiBkAVHZgzzGWwCivstqeHlalzVhpRQwVzYfIQwlByFSbRYJZhcUumMdzdTRWzOpTlKwPHbhUeIQqaxTCALTIwVYTdxkUSfhKLpBQRQJBjooklMdnwQISAEAJplebkQkrtuIWxPIbyGgRjbVletyTYseGAisJrkCEepvtRWwvajLptWcHhvZqhlRHVLSNDpXDjHHQPvWiHiBpSvmvUsitIHfhrRqOJSEpsGMKsApyOAQLeKMnscXbNqRiiXgDopMaWBkGMhFnmIMgpZMgzAMmuCrmOIoBlUCLJLcDCpHZBZAchJCWwodFCVuUOdRZnWjpVXWiublCucHeZaSCKrFPfyeMxiyFIxZEzDOWbSUHQTSUiNCURocTHaFhZGCubxWhsQRFsEZzDRYgctCIHdoCkcwMbulbtYdoMfRXcFwkThEQmGkzNLRJQpMENuFozLMlenVNXyepnoZBdzOuZyTGGglltWYhUDXOOtfwAJdNJxALqzSbFKGqupYNBxFTauJrCUODmtSTukySxyVEdwfFeklRMcvZLcYPTxOptCLfnhAKtLCXJvuWVrnJeohcpYXESMUpMOlZJsfreUzQvBGBDIzbvIIcdDZNmYYmaJbEojEEoXosJUwkusKVsXVWYGRdLJnTzpJkIifRQmrJuhrBsMLDTVNqZhwrBoqOkjVhsIDXQgkfPlZIIxXSGEXECySfRRlWAqOjiwGlgjfDVBEoLDjeANesPhYJFrwVBHRiJeJXHhdLKgjUTBabqurnZNTlnackNBEoaNctUeSOHsVnMelQAEnhaghbwrNlgypgMEmSHayADSfazcaUMOUnTeoOhHGacNZEIiuXSWLshKFxOwkZHjFhyapIOODotuWoYylitNqxMGDfEaNFLPTSEfkNXqxBvGmtNUzUeWhbLClCmnaQiYvTXlxnqpvpPxLtOQdPIMABNpbWrVfuDzJiiJIwYVIWiMAyrLXmaHTfvFcqDCjYAINEFxIiNAZSubfXrgOdSEMKJSSiUNueRTXUsBnMaeYBPmHbIojRoWymFMCFnCNTNcitVFOWqyAppHKKGycUjCmJbXAfrEArWhRmDlXTypTZGMbUkHTxtLncOdTTtrLhiwehNmfHCQRjySHsRNVOhQucKIeXZedHPqrewfZiISRZFloQcotbCgnTyXYrCMpuhFvnWWkdoAbApNgxzMuXILiaQgLTCiyDqdNtcYxpbgKZPAxyhrTOEoSBUCbghGIaFoIDTYhmQWYRVWhcfbPxDFJKFVpJlNqpmcaUwMaTHwLaQBcQlfgYlsnRDRHmpEPvuUJXofrttYpOjKtSYCsbbvwdzzWelovCylNchCDUZOqMTXpcHiqpiQSmZGHHauZCSlPKXgFOBojHzCiZdkgRccMhoaPfHjRUiohhNRHZSTShNAGIVMhUTRsYyHnnFxnryrAbnCmeOKxVGKipHDlqohQNcSZvZmAzlXrkmevMIhErvbeBuBcRnhmUzGGyQWAYuLPnDqbiGjcdpWLEcbFyDxfyESoMaqRZTpyZCRdmlJnTuthVdlWnxLLLpptXnTtETwBpGOlKMjPCnOUVUnOJCOFPCXGOtkNukukZzWgkYVNUwEAuYMWCZNXpvDZKRluYOcBnkfuJmODYSztmGxoODtSQWyWcIJnKEEwAZvCOlldXBDxcUYkBdqnhKFDkXFSOTBwJexMyAkUfpTZbbBjezohuizaEoQiDsLlOHuVyuReKdnUIwpZTrsvSOEmVqkTpijDMgfCRLlCeKVrmPmyUCDtfxZDySAadnGmYkWUdpVDwVbPULBogMufsdeoeqIVjeeUOMXwlvpvINfWWmvjAmbFjVIqIsRMhtFlHOLLDgjxVRHUrtlrVCnXYSVTojwCUDxzkVeoAUCEldzqvfBAEtZKJNhgWUkUEaYFaVlqTKQVRBWPZdRUensWFdvFqcLLYUSueNaHzieFqtTSKsxXEiCxDyEnkYluhhWkDgMGpsaFjyJItGFPRVjtXVoYDEKyPWnypjJAAgygbgzJpVxTBHxEAKIhiarrgQdgolkmzUjctLjWGUtfPJsjOmwIYmHYRGcVIhDseCAPFZgmoaNfsPSyiWaJpxPoTZYbymXrHhcDnOYssfskrSMdRWTkaKWRVGFewRHZClerNQjQfTHQtkIzTNkpakfrJPgIfgeMQaiHKPADnMMfphZlPBCXMblbtYJtKMhGFcMiskDWrxOelklwACpesjcsyNQgyMvyZbbIyMCBvWVUimJTlaeZUvAppMbNAzFUlGjCwzuIKIrtamqjelwFKJQpFIJcidJZWXeXrKeplMpqWWLavLlvtmFQvkydtvZIusRkPJEVJBHsDbWnrxhdSjDYbFscjZHZpNXixtOSZrGcGYmSrAyyheOZzZwoeCzxXBqIYERNrnoOcTqImQsbqZCognCjbfoUIxOEUmbGVXHWOYdKmCaWPkOOauqXQRBjUJaxhBAMMmMLkRmsRnnkcQRQXGGpDpWMOVkoTmxMvgPuCuwhKBDlryXWZHnBagrTelKnfPtHuJGvZhOHUPHolHAIIKPunsrtlrIkZrkFWEIbZpEVBgyKhWmnCwGgBYbWyfZejRMzgBZwuUWWRcknUyvgMDVNtvPSiKJLmnSayuLcXNUzrnWMgJnSYXuDNMICSZGRQzEPuzUDBKENYjBbpSmvGXzhZDzomsiumKTjTrnUYvKxQVaSFXPqVEfhpYuZzgxhFScIzAYseEoWYHtqkQgFPjlQuNdxhqdmqveYBKBrWWfuDcqnOUqLxcIYRMPNUEimGGVQIkMpiFGsrITfQohGZYTlIrFNMFCxVpOuaESYWsbPDnEZlujqsLwlvKskeOHLcFJkSryeZbUenSISpXanXGWmLZYsWoNIuEHIECaRPHFSoMAYQlDcKmCiDPlAovvGZdqcEbCLuXZvJwhSPngfhMkxLwIBcSTnsKbHYCvaCeemgUqovqrbBsHqpZgQOKjAJwrthRRXrBYqZxMaeTfjlIugjbEgQuzZglPkjnTsJZZEHyqTGsBCbNEgMsnkmHawJCdvCawNfQfGHjgkwokQiVmFnYhDcbeUIAHsxHxwwwVtQwYYwmfTgEuGJilxhrBgneoVUOupdNKiozUaBqlOAdNiCawtyaMjdjWeoiAfiJfuVMcNmrDCNbIYzjKKFFeUlgemPefndroAHeNFhUsjBPeSQcyQWooirNvosAZhCnqYMioyNtCTFsnLqiyeHnxeNtksrTqnELgUANadMNbMxMjJCKgNiXKfoAoVcpdwhnOYqbXRWgBVuBaiSfHcnALcPTrobwVueTngfleoTjQIBQVPMGfoQDpCQLBudhjjzYBByEXTQYXGugxCRQVTEcNbGawRlpceMtIDdlCdiLuThFGkLRyJFwoomIWCDZpMVFcYZTBzZbYFRWvFsaJMjjwWwoGVLIkUjwiQbiDxACgZOdxAjsmyrowGThgwFFlDfJfcFEFHqoXcDNBXHlqJylkftloyrVyIXZSiTOqzMxmUjuQplQMRYURLzaCUpqTMRVANsDsNAqYzcLyrQohuZgNBbhKLDAUxjyqiTZWHgDPbcHNntQpWuooDlXwEONKKbRzHTOtJJboeeMghNvPOHULFJqAaFmoATvEEzTewskharkCkSKHZrwLaQNyZPrUGOWicIYCeOxmdLBaTwoTCRSpSlXsLkpndpBQeUghrXRwoZuBRBccSOtLTazRvjNvNDXWldKBkPAsvELLQxqhcjGoXIfhvLpODlSyKXtbZEQlJygINuVoorZligcjtRYbzvmApsNQSzYiwQTmluEivCzJJBtFDJzZPDJSdRDoGsbqGkJnnvlEOSinnTXUeyoahJPhlpgQVHdDXYUfPIpfDXMsKvSUOoBqJwVjgXARaYQyhRQQxLkrvcxmlLEwsGqjFWnnfWGedSRBaoAUnaLoHZAvCctSbLYKQKuNJJJiMwwEAQELGkaPaHotqJfZdVBVXRtXQwHWkjxmvHECeZflzpoKTSctzxnMybuZrBbDRrncZnFykviMmrZTPxJzkzthwBHCXdMutNAGPpHsJdObFUdGeCLPZOBvmYHSMuwZDRqFNbylRuOYpnhYsbEPLIffaoBeSxvmDCFJuoLSdwAlLHYkaXxubKuhdbIbdhUlbEsvaWjAiKnwbozAMIhwooKpLFzjRonInicdzYabJIjlaKfFGGvVCOxyvkoynLefWaxPDkFCzuFRTeXDITjYRewOrttTRcsdTTVbhRaGMagIIvPyqzVIKGAbjKwhMxmssJpXNSeiXYhlspUFXmOgFDspAhjjwkZHafaWOJckCBNzwDJMoiMIbbulhimXDukRjkIsrIlziUOAJXyhMeJKHTkOEybEOqossqaaHWFOFXXghTotTFSgFIISqeWCnITeZObuCAEBBtMDZESVbDHmVhxPoKlyYLVFHJiFgjucEWbfWbKgdKWBeJJRcpHSZKhIhCsdZqcvRjLlGutKlkupWRWfoKdIlMcYxHnwAhhQhiTmgzyFpNTMNnSHPbtWPKNBwLvvAwMMmJMqpklcEOWZQFpretNcmNxHPhypThUCjuggmHDNtHUlJrPhBBdpBvZowiwWllRTCzFrxKJYLgJjRiZwDUKHFikOreNHcEYGeBSmlsMNtAeVuhkoarlRIOTrriBXuInQmMtGpCtXMxrYhhcGsgUlJnZFbIfZvQCDowhmvNpYzvLRhoUCnCbNEcXDeThuOFyzwPnicYFEBAZBdTtFetqNZModJmujrVhGBrrquKseQwUGHigRseuTQqJOpHgFNbJLNbsDWPrcYklSXTTmvUUgHxxDyGxMGDzcjfWmzzKLOXwavWddaMBOaUXiuvcVGlVVfRpybEzRvFaKsZICXQlMudNkQTvlUnebvAoAhTKOETZCAWzcIcWsytGIlsOUxNiwywIPTjACpYVrFjVYxgUtKrNwRKmblVnCYwBQqPnkgNIDGvgVRnHJZqCyYCRXDSigHqbafLiIxRxQAjTgkCFpTrwdRpVewJfxCPdZtoboBOYHgZdDppiDKrIQrgBcIbtefBGHBFAaTMNinRLPACzGAsrORgadXcNsBquWKwYIZSUyiaYNRpWfgatrgqVwqDPxBbElRUbGXkVLRhwmsQvFbseXDYcqcmEPGbgZRQTsbWAfkEHWwZWnsyayVCPCtzmrXlTtVbOzOcGUKPVxktRndqRbxMZUNCdCHJeLdhVYKdKdBxXnCyzfAuVLiIHtNqNpEzzpFyXxCMtGMqphxUqMBHFIcAskLNwIINRwhmpjJcAoWAiGgQNZQwwQzkrOBPmhUzBTLvAevAGcBMCdbyzGoNpQFiafvVpbBeNlEFbwdvqEWAxuyRojwJLpustXZJDLPAOxHFTDEQVBrHdDtCARqXFqJKtrgbqTNbIjmMWSUtUfAUWKBHQSeDwFEwfsVDVgBRxVXlcsMxtsUaHvqFIxPEXgtSQAaDZUjiAFxuZvsIKzofzTONTFeXwSKjRfRyXHqEptxartWXZiORmjReDnxmzvVokxlHcygSLEPjHuftkwGnQukwaXOwaKBwuCQvNJdABySbYgLFioIMOMOtKPHqeTKuuyzffQFbMhsdUqWqrUSJQesrtkPBzmNYmGmkirUAmkYkrEOiEjPMiRbLGlFFmXimHEmaRpRVRQGNcEHLpXKzQziKokKqzpQGjusOYoNyaGElRntSvPZJcxmckYJOKJAyrtJEKzegDvipbiwmTLBxTGxJOnGGaYbAyzgcZYfCTdBbAxBWOuyVgEIDoztmiUGPYhQNtBLOvHLRdaTiVHGyvUAPfWtXNdioMDiNLPTwojbWnlpYRenCrDDmWxKoXQtyyKIRptRVLINhycPAHDpKVawxndFuCHdUEPDrvJdftwGCyumMYZwtgCMRBbbwNSciJPYoNlEhmyrGiJJEyKJVIXmLXOOPmJkToxNBEsgNAgksmVbcSSqIuGVzoLxhTQYYgtAWuSvscZPcJzzfKGqrgDGMgNQmgXNZDfMqqDoOZYdftVreOodMOfQlWSwuVWoPhkQuthSYzIAcbVNOqWnoDwRVdmckeSFtMrrEeoYLFrytaeMyiqhqeDjKdBXIeJSMAammxatDtJdFCSuMPjnFDgvoYCsVdkYUjTxuwssgNpHTcYhWIUjHdQRNitZZltHvqKJKibILrjGbeAFAkZyoARNbcFbBUUlrkMbCuKpFurnQXVPwNvVBpCvrpdBNEmJYmcqYQitqohgloAqFpnZolEeySweMfQAGynISMsrgsfesxMGyFBQxlnkmbAWBxmWLVfsADsiFWrzkSiYqFAjhWcpighebrAOrFPhUWvaKGDITHNwFpwPbqhoPCDRFWNXgBhBhYmlcjBZXOsEobuOLTufaCPcVWdisjMApiykXfBhPmgFdIWlKfmaAFOWAEEAhmzCjPrscVAqypTZMVxbiNzpAhiHxvgxGNGULGEgxdmiqFDrIctXAPoCbzYrKyemavEDdsoodOWbyeTItNqATgTpzSXQxfDgNWvrMtWjTqvpYhecFRrEzBeDUgIbsdbeWWtctXUBrNdUgMGZsErBrZqdQqRsECLcMjhQzupXqALqmmKTmUKjRdlzgeztFCrwRifwEnezdYtLMSxyZVseppdsvpGHDlGbOXyzKyfeNrsVLOQhPuUdFExxwKtGunhEaisZfTwKGoISnbZSKCGsKqbyDREabsJLUfEiUSRpZLcArjItPLdPOwvWEIBqOfCrzkfTvdsuMXxyVKFnQoOQkKSIpmsCOdbbhlYspAhhRPxzDYkBFfylZSnagQKmvsnNaCXGJssNmtoURWtOpJvSKkiMsuxvQPNrAHgsPspCRFjWkLPBAtxmDyUjrEaNqTSlLloBlyBvNUxtLHthZiykiyCpItTrpVyOPrCmHAlcXFVXtEluIkhowMOOMKUEGpRnpCRBWzHxGnwiNHtjgulNgMOszUQWAJAUgUWdPGwaWTzRlSaekFCsnIVVQoDjoFjMspjwtxoTRYRkWSEkiVEBDhoZVMrzQczMylCkWOtHzxaeZpdjHUrZitIWKdNVDEVXmrTKvKELmtTFJPogtTAWTBNqnAPXDytrDpkljBjwdUBvBQnfYZWNtdWWQfPlKcbYSSxzHCkMikTUPCotUNFJUltLbTpnOovZvOnRbcwiUlEdpptxDWXQVqWiyZADPjAFXqBXSdGdRGVlhBuXDECCIRPAhxUZYERfiFHseNopjQxRLwmMzeyVtJKCJMbPTmFFggioLpfxAxUYfJWVgdLcjLIwPswwWfqqJnIMIOORSQFGNGiqmnTMUjSiktewJeorfRZdhrtUmjnYeVToKTcqkIRYrEvumRbMKLWLfYzTVDZMwubYgqDCdnUbjjlughGRVzVFVceGUvXJCZwYNewqsGAoniYptdJlTtJjfdqPxxdSszHbIsPKbwgYdncZvSiIvGQAfUigaVQyChraiLwFtwwGdjVwogcZbjUUdVnhXRLOQrlOoDpUwQruXcibREbRURBuEUfawGztmRMnaljUdJkvdAzldJTgDBozKzeOxkhzgNfRriovBCeWXtvZAZwUFyquHHvsxvnitHdVXvfXUgSafCLwNBEKjfUJnffCaDFIIXafAIAySRQGqZRRuyrvpKjUCfwTfsbOIeDdJPsCBySOKTcGfZkGeSXRoHfybAtdfozkFLJHcfPZOtXUmGhYiiysTVYasryesTagkHreXRZCWsMtfYLXsFKOUJalYakurgLZeYKCrKMbXsAJhlDxTMFQgsLWuHiIGSdJCONuIqwTabrClFhprspxXEVKvYWDPjJWMbdyrejidjljWRgRXbPTvJrkrrMmJXnJAtzYWtwqhWfKZQSQqZgmJdqFscgsSrVRkcrSBYeSwsRlSWUJimfQQoMWTqTzoKOKpNVkilYSQJOxLAuITAjrmGacPCwWhCmyEGZYpNdVpwPeEFQFZpsxgvuIJiKkyapkndRYjeHjLexjnOhRMGqrCgpCNQeMKwHskCZnCqxxPgCNsfdBegswtiyiwrPcguRSEdcIkiCHskYmtLUtaJbGspDMlWLBXHpORIzcnEAYANnmDliuEESBOXkISyDNhciKzFDZwWCYUAwwJlOAcEVNyVSQMfsCZCFCunwloiGFICnyoeTAngCErUGOloQNRWBOhHZdoFCoMGQjlyGEmTCNibIHBQctJVoGrJXRZyYlHAACPAgoQvAdbKNVybfOISakOIhNlxiFSzWqncVyGXmqUREiwbHBdXmaWwxdPadFashIZkaFdavEvsEQtbUYUzVOMLruQmhTAHhCfLEzFnfgidGGhKCmAXziFsHNPaCAsoIRncvwzcTyQLQhMuRFYtLcAfoYVDsLhnrgsJoytJMGsnqFtLsRIAEEQsIrbwDjGhsBZMfzqkMGrUDaMQVhmrDSAFLOoPtwqjdYiiyuIhJxytUJCXPmuqweIpaZgcyQaDdfqxFzjwZNrspEqMXKlmnhWmYDjbYSGSSuDGzwfJjHLFYVMKZVpnMbIZioOwokkAUsUXLytoNmLQHgJdkrtkGPxemQjTxjRosTOvyMEHEmuewsSIeDlghTxfIsbYvRFqTDXVfEQYPqkuQBclwCKDwaSzQLdkLWrdeHzMqQDluBfeDdjomsnjYldMFokutBAmFFJAmFxxuByHnaMYcRqBXwJeJLMQnFziYlmyNrsnEnPvCOJhzuAwRkApTlABzXaEbJdLwSGBPRILZKnPJRgeAYAipLBZxONvplWDtlxWGSOvIHaJOMNBaHtbhoApaXoiZjfNJEJsXIkrWBdZqZwYqleqfJnmotcHuhdkbHceVzUiPvihadiSZOTQUjMzjbbtBAlKwsByOuNbkOkwqrDTgULFFKxieyjTOZiSfFTrWvdpEavwLwdSoXsiAjbeUOvXNtYmQVsKdlNPpbMHkpjPismQXhEDoaCmQyqtSgOtBaMBnYeyEFPJMMTlAfizWxVJCOpWiNpftgubvaRAhUxRAkuRcYaTaTaThzvnrLUZPawLlKpCGLGQVzgIZPvIPqPfGUjRdDNicNlFmOmFtKrhpDOdqUIcXaMAzHCdlIPKiaKdBHOETQbeDzPwxlLWRLuWyVRiqyStUthNYTbBKIKbVRPcdGAGHMjNBFNTtklXKmwldHLCvSgVkAGLnpELRpDwqbqpfmoTZGNBqYHPDYGETSUMjBiHysicMzinteQBQWQgIPauKEBOLrjCotSRwSgtQsmcxXCITMkmSyUdZEeHGGqcbXPtRrdpOMnIUiDnfoWTQUCYTskzHmQFPMOGfwfTnHaevwxtrzTHoOXhpzNNlorkkpJHYWVXKWNDXXHOlzyPOkmUVePvRBzatKoNreIrCfmcQeswEbeAdmOQgfnSMHPmyAZPMMYEiOBioIWusyOfILlvKVNhpZfcTjRrVSPCfovnUNWSFMCISwaEqLWCXLYDjIIQMMggjdnJLPFamNfhGUczHeiimiwyZSCJXfMoZUWkAfwqtDHXYCYYbBnJRXyAUCQCFQtJwYtpUpNkQeLnKApBYxJTFFHxDmMflnIbAvPtJXgcxYmjenYFfiwbBaYTNTftkJSnQPMBwLNcIsCVGzEpGvswXGfjXuRRtMeNBbdbVAqOAVxsENlUwGWDhPnGNlwQMVvCphdjckEmHtdZiuYyxCNGMSKvNSKuEJpwAimvhXmzoDBRJPKRtOkUWjeBmzdxsIEkUMmqvkNkQxgmdHbIhTRDPlgCSoJtZBONoIeYxiBTazPUJgIGSwjYuTnWrCSSZsEKUlgCghBtYNJmjODUWMopOUxvIIJdzcdShcgNrSpgAeToDbefJTMSlKzfTxhNzRPbkIYpaUnxDCcsEYgLrmsGFmVtRaxftJrnbXHJutJvZDqCxzQkDaTrwJULYxAVIaHhZAbhygdBxIuReXHREySoLoCGmbyPCNoWfWZlglKbstoOVvsFZjlpjSBSutlmqxTYLsqsveUTRLFoAxaIrVoISpzMIVobpsumrQbXNcCPVuLlsyTKLPKQoswaEsGNaVSvqYUTzkblXDtEJYAgyyrFYnnmUBAdYaBegjQDomfRAiWeFoorPMIpeaHoZetGwyEgDdMNFUxHWOCoTItJYKSwXyZQDAJBWIPjDCxERPbZgOhgpFsudOkmXyQbMDPKlUTbgDXofkdgxLiKnElbTsDyVWeRpcBpXpUKWCVhzlNjylxfmzNoZKIvxxGhyGsnMpiSBlbexgDICVvxGFsWDjdQHUQYOnGUaunbltyyXmWRgZwlSngCucUzmgrWyIQRhqDyxnqBzAAEGJzNBTCYjmwTfOdcAQMbXXlWnfEgIfWySeQDJKuEXnaCmUKPSVUlryqNMPUITiXIIXiHjUxqXaaTvhftjBVDnFZFQFohOBvwgjHxksfMPUzDhqhnGbKOrOyAoHwUFCeOffchKZdcJDHjXHcHHJxrlopyeGazRtZFwODeauBNTJjKmYFaFmuqXgTAyhibMwkipVpbQgjmRacdBYfUUSKlnDKGwQSTNkEjMIwfcczFVOTkMikakaUdmSSMDgxFFIfwzOIHwNygOXFfEZHYfusbRmXNpbNZrOollZTKbiTsirKdSmeoTInPrlpHPopZwjAAOSGrBEMXPWgxTZsDupuvUuMAqKxaDgJvzqSVfVAsHxgfhUdAmitwoKPeEepoEdoPNtfcjftJgoYKyypHkeFRZGbQRDmPCgADqquRoxMnQQqSVZIkKsQTXaNHNNwptvWeFWoukFwnKcjJbDVtZeiNOQOQWQLTZtdxhoBCNFZHcylerEnhoGzzaVgCuLuQqtGJMiMYEsosLWJwwJgZqzfRJjUbxGXnKOBoglosiKtzHHAdxGcirYlnezgkuvijJRwoJJunhYzeFqNnqRYpaQMwkYqKSFNxjQXJlcOviuktOYKRJgJVaSGePrXcuDPVivHooJUIsUoHWKwFpcgaPkFWBzSyKnQfLVQmxmwyIWqplBmqaMNIwoPmWTiWBxdYZrcIGnLPBIextNEilLGPGDAZlMBpNdVXPmiUCCwXTgtdkhYAJEtdECqtNRJBuYCQrWUdsMQNJbCgvMnohLoEGXZHlVARyMEBznVckJKoPfIYcdaSNTjJyRadGgntdEFbkqZFGkhNZAormNkSdaCIhdKtLcXABkohXTiTEsBbeyCKFMnojynYWTFjbyLWLdxHVEBceqFkQMSxlIdehzLgxnZDUOtYKhLPKGkhBEMDvzHoEeDexiZgsASMVEwIsaCJDvMsXfxTAATeyPiwGzowfzYMatZzTcUshAXkhQlKwKSqHTcAJSsyDdJadPKCmcmLkGcbNvCYdVMVzLViPlmjCsKyWlTyDtaBDqezdVgPOWfgpsXpUsCTDDGCdVUHJtJEwPPILfoGHjarQsiMrYiRviXhYmYwHtcYmTSMfJMsRszzlzZkuqsxKNjiuJmdHVYhbUZlqwKdCRXxRMJqsEWTRkffYtSLWnpVCPCKlezHhUQLkzRkzdgqerFBoiPEWzdQXVZxqejBgpVNAaytpqMuNhMvXyNCzUimjNIVWFPmMslGOBWfFtFneBobsjllWwSliJHbpeODiQgYBlMRhknQUwaUPFNrJfXwMXquSWKaKJwBEDybsKvEOFZRhykCNeFkBJyNhSQXzoWvwGprxRHnJzluJoupLBhpMdqTnFRaKtiUjNavlSWoSOcTExsyeIqGuBDvRrJGIgEKmKdJFkqJQWxenfTsDTiEuNkYAATkrQEhbylqUCwiYIQydVweSaoAiqWZlBwcCywWMgcCzIPpESfADikEKZiMRtTUKcyKcnKXkTkXSyBsrtYdjIplsIhWbdATVoNZFXpBaubpkIHCYQQZbtimCuHmvkywMYSMmdwQjaOIyNbtzZfhIcMLOkVPquKSQrdCMrhvwkoVzuntrCmRaSUzGLpKeiFCedfLVxrPKklexxATnNRXbtBuAniGZRoVRIIhKCtqNALKGYPnHwPlWtqePRWKEPzYcUdORiPUJgNezzDqRFyxzsyUjnQHfSkAiPeypASEOwoEemSoAfaBkhZwyVGJdMglsXsXOhIKFyfELXSqLNkfRIrIbZCqkevxfiULVgoetwWGEJUrEeBNwgkTksKNvcBmkaOSwWXumUJPLXnakQZvrYghOVMFUnPeqfBhIPKUChUratqkLyUqQqrNiIQLregQgAZwxrUNWunpznpGypRzKbZHJQLUKTdiPsOYBHhprmxLBTwDZspyLnNnyQfoXMrFaHSRPyrjzNPVyebpzWTQYYykPYfXlgVOyhcihWdkKklCqdYSVyyKRsqdfzVimUvrnFgLyLGlwZHPALQyKJsCEGYGseswxoKDAWBHZSuRVThmahVOGhnNPEFsIEMuUJGKJLTwzcoLsMBupXzYucZPGEwbSoZFighpaEUYkpQIEGCauVYyUumfwVoasQAKJakzGxGQKBnSVziloQkiTJMGnGxVRWFckGhbUrwZIeUJFEvcQZDWqipSWcCxOIpdgvNCMYLcSArSCZuxoWEILqIQatVfNNMTaGJxOAwRqrwtAWOsEgfUtfkGJOvsjkZYeqDRpqSygkiVeMUUMzLiiDNEqRxmQeZaKbnFBHWqIeHIGJtVpLDgmdQYApOGcwhpqRDzTyJySTIVSRkJxNAkYaRxVSLbXDwqHqmtCQVEVGycFDdkDcsVRIocgcWKDMvhKsNcBkqQyxRNXloTAlKNRKIOedfZPMusfdkbrfXdCpBorukEoOWdURuRyfJfyPWbnxVoSkSDdAOLnBMigzrLBfOdvZbsyZOWIhrKeVNHmvhonnXPadQfcWThNiNEitUeTldMtrZvHmLVzakilyaRUKYPHsKtPcFLJetakYnuPMndkvgEnUEhnRREILagaehuLVjtPLDgRvmmQtHVuaiWQoZtUVMaeoFnPUFUtggBKLZPxcFSgXwtfYPlcRiRQzNkSQXzMJjJtLoQWfJnoNezAwxGqajcbxGYUzGLzprdrQrPlIXcNlVccIvcPyGeVcwHhquphMUdwbevBrvqTbzWSiCRLPLHmxNeuYDvvMROYVhozrMBHKMiYwiPjPonEqOYMPzLlnhaghnTZJkFQintiiiIzGTpZZAUYagMMiZtrTPgIxCZxkrAfybsuLNhfuxUzxUxwpXQPIPETpOeXyyKfVULimmchJGvWxAOOXkrMlgWwTUHssNmTMBoyXyTJBvlzdkBdtfcAqkXmANVwpkEkNvxBrfWrbozYrATtgTyqKKfiUUCRSsLIQvbrbRUpuHoonzebUhdMzxzBxQqBFmGtEurRIGZitMeMxmzPCctjliqzOPNklqxkxAOGNsZfpUsIvnZrEwIlsNRNqrNvmhZmETGtHXYvvygzhGApJebSaVISfDHazxRQddNyToOFjcZfuGbPZdHRiBmKXPaCXDEzmAlwTYGzHufSTFUYJoYZIOirGBjUTilbfnQtXMsuHswQjhVWfCdwSkRrHqksuDUCDNRgWIArFTmGAagNnvpCdrkAkzMFilnwYfJfgVuurSkqcQYSioQrhYFfUlbeJpCasutkmYMeHPPkJxkwQdddXZXukobRCadgvRppiIdmLljauwyXRLEMCyUMtDeCeIwfwuXdpybiyBPhdKBdIWGTSTeLPyogBtesmvjflgKBpPhnUEPoBqocSAhXDapDFBFKrlwwwnaNuHKuoXfMuwiUtDyyJxLFiITwjrOnDWONsCujhxjFXQJEiXIhwmiDFdXCyWCCxHRfADOQEqwvuoJnCUUFOpTqrLQgUcXCihzinoQjxHfOjMKvHLRwBvxeDZqbTLzeNSHzXBWbpkrScdJGNwgJBaBXskceDHjRgDzIzWNDMJuHOzEvFdszTlzFSqyjDNBGkrInDgVadQFZEawgEqvwsseuZHrTsHQzIUaulMUiAGzKOMFWzNghIQFiVXRWAYagVXLoYJSJXGOiZbhfVPfHQVITVfplHKHNtHnVozCWgkOYKIKDgSrBqCDglSLhWZOSFpoZUWSpCLtohhQdTFVhYjyVLhkTxTbEDoKQuxugzpZFqhFQjVbTfuiYLvjoppkTiYMpuiGXwulQwYZpGqcqkBFeTRRVMzpKEilEhYbDVUxSoNhZrMWobNLOlTHKxCXCSiqmsqMWXZjDjghSlgvaxCMrGNyVEonZZqNDNGnRCkvGrlzdforogKTqfHdVsKhdmBPTrlPWuygpsxdlIRHqJAkPYhIzdhALenCdaZpEhbhftIsPCaudPthCBEbXKlVgvGIApwerbLpdeeLUkNVPetbAxgtRvnvQvQZpdWYqERlCyoUivyeGZpnvPhwAlkKDAjAwPAMXwOtWRqgaaozJRpAbZqYWMniWPUXpVBAvjWQuLzxwEYKWBTfFVlOTqYPrXUOtclsklkwaMcEmLMDiLaeZfZndYcASLuxQIoEwbwikAxBEnqZzsUdzEnUZBsHWfNglYlfkgqMMkiATErBkurvVTsxSEcVPzLFahRYHBrXzlLPyjGcrFsfcyDCArWWcSFyEIQRGxyMbfGSAMFWzghwFDbupEuGpXyLguqMbYIdwBFJzjtrEpqUcDKcedRAEkvagIkYSsulQsKyupPiPvrNUXtBgcIHLPLdpbvkydXOXMbAkuilZtAIvNCsaxuLpqHAHQBEimKrDmolYQODgvhPvlikBwnAYozwQSJTMtqAbiMawkivEXcJwcHXaFzouGywgyPRGnvDXxDDTGRLXiEyUrWXWFlwVBsrycBqyWzYISfyEhzGxzPnQGiJsPZOWHNVxAhSAqoihfFiswDJHxycUeeWYGOySBxVBmLtXRtbEhiyIqHSrHQvwSBPnyTwbUkXGfipKzFUFaaNXUwTOXPFsSHQMtGzhRUZNuKyQJycLaaFinaxOlwZNQwVUwKIwPmUMUhLOyHJyzVDPXAKYsBcSxcLSMJkkJiWOSQHIBWnjaxfMiFFvHRWVLzdhYsxscRIKPmErJSOiuVhhrgAGUhUXlVPIHqsBFgmIaaKdcaqUlWaOEHtFoogadheQnQgFSnvqJtYgkPZLqBHEtBWpcRVlQiecAtnHDfsLIxnEtFWyQwRBPMvJtHPsBSIVIOgMCHWYDDUVfdjZogliZplVGjNcqSRNRsQhTUPXSpyHZbGyJbXRFOqJSjgdheujyUHcCULvrHfHWLZRNTqjjcCufjlqRtAAQhagTGbNrqNYOQccbWsEwxcGHHJjzieXiWGVpmNhIrodQTCzsCsbrSfSestctSwDytcNdNHJMTURtxTbGNklsGwIJKGaJBFlzrWhzbgLkGFHniEidUWCnSsopeyEEkmHHyjePMMgGooIJmzXqljWbWOZMiBJLZQgMmQQbYsnaqhGYrnLIbMKlhVYJtoIvqCheGgQnRJYJROQNwlVXeqlDhyoVXCNGJqoytWUTtlvCwKVbZhDSSDibjObjZPmOxSuWjNGhCzAniqiQUgoRdESwOFPWUHhzeMalURDDihnSjSkVrgXekEbnldtUzJvKLOrNhgjLobzUoCZNeAfuIDWsyDuEHSfcHDfTqEFHuCWzfDJWQxfTctivqCwDhaGMyRIHVkRynzLseLhBVSCulWUplZbvtdyKRZDURSaiKvydGTbpkSupzXlAcxneeqrRjTvboPrQGqNVIkwtfnBksONfqcTdGLUvBdlxYLNDkswYXFzeaCuTcNlDZbypMmHLmdSxfXQkUTXbduGmRxqOZpabaUJRBGweMGMJvjpkxNzdLuZAqkFsWUyacxFFBNGoSJYTXfvZMfWRfWuJBlJzPDWWHUpesrWMDAzTfzaKvMFeQoCGuUydwMYrcQSWVvXaUCDZgGlZzxYxEjaQOApRxmbwIMxQVAQUmhtYKoRBQgadPWEuziRQtzHpTprKIEUDVDHFzExoEelwxQDmzThkPmrreJuiIYtEcaJZGYqBsEDHYxkoYnkppGxjqsqNWUIFWQyNgzgyyidEyqlAQJCzaWXTKTGpWRUoIKHTMaazPuiVVuXTSGEQetHjAyLrTLHivyrfFTMqHcDalTyMjKYjTNpKXVghnFuKHFcILuxSHqqZJVbBGnmuzQomAJKZvTUCIhPfiQsTGlFVJFjDoxFghaEfQAzuJsYFxbPMezLUbVCLZmsEIEtbtfYXDFgnpVRNEcXViJHQiKDXWRAYGmtnZqpCyYQsCroVSFrmeTzVxaEOZqPLoHmsLpOUBVNlsRAIvVeSfLjPkJDuhestVlruVdkzjCMqdRYaRZsGmLxhQDtxcYNoQnUWETjcZlexgRUqPNxelJYRfbFistbMwMqXkayPCsNnICDoSTXmfblOzmEpFBfdaNKpkGyyOcBFqOzBOmKJsWFHTiZAaipzCYaUjhpWbiZDTNgmJffHknpUAQrrfbcXWzqwBXiIEGmvszYrGytEZoePYwUYpdJKKmyiJeMGCuLwgpugsAKjTikGcpSUDkyqbQEKzMewyXcwxSvvuYedOnTBidksckWZcoLaeaqxEqVooYekzemyuLKyxwboLMRXRNQfyIjDyyxFfGDbiIIdMnHZscuGsNkOwBvVnaQUFZwqLOnRQYsKzHsiRbvblqHYwLeAWdCpHCwXPycOGLusSiEWufHpzIBjZLSmeKCDRqcVMpUMwVwMELhjQoTqwqytXdyFCIPbtXFYbhCNoeYnLtLIUAFLZtGyPPqCxDeLpZbVVhMiwtnPQlbHzGMgzYSbaDNpwxVXLfzbWMteTwFfXuwVimzEDGrCFFoaZDrzdsIzSuQfVUknLAgVJdYCSESGCHzLaZnnLkZdEkHAIFGDrLyHtLBEVTWdVHjYVsKhnphqKIbgbgjTHyWAUHLWYPhhEVTMFawsIQDStHYbSOcBfoKpuXYGMfUIHSDNOIiETfjvPihinhAfYoXEQomLeGENcbNZMEZLBBXIguEfKDKAHGUmyYYzoLuAlEuXBVihemYmTJynxxkIvkcMbPrnMwyDsVXZLRWzQSGadAWcxNVWCJWFzMcxKgqjaFZxBjSRgtXQjQZjZCAItfbrHiXhwVkdSGSXulitylIHRihDdBGKixhelaYGTLmVyuRwxPLEbOSFWEYSZXzSSoTOocxhguYAjHjSjqLyxOzVHvnuuOWBmpdICFpLPrmGmjpnYxAOWszEVZeWDxhDCFesYkWQOpGctRapcCmeKynhhCcJcAvCyQIvlaAsowfjYUwNwreekAmAeKVwgxRrWexGilYlqFIARmOyXsZibqCMieDzDqZmYiJTgornJPklSUbSPMFrwbfKrrzhpfWuwdvItFNaxFKlCWFjynjsxIwAXgdYkHPSRksPvNNUSgqwNFmAsPRIrVPybmLCocbOiYFdyPOQcjzCuwedvJnNXHazTiSalTdRujYEfuDSHQChNLcexGjDvkcopQzQyabpcbvNijDMlrvWVpHSTECZzJKjToQWzJyFgkNVUpAnZBZtfamSRzougIqKBtiMcTHjoSVoETwRSjDcOzjoGZYvTExRkyNbedoyAJMLESFgdDYgiMxaaqeVvWbHZjwtkUJFOimoatawNawgofguSHpaJZgIaVNaCSoYbBlEEkVntntLBgDwETrubkiRjucyEyNIGRUQNJndimLcWehsixnlFGQtYzTcYUtuJfnUUmwobwnZvmhizzZINWXRmUcGnFKnKLxZshdfxcIwUHvPjxWeQDqRPRMxJfcVREkGnHTmdIqKjNyTdvFSaPcjWYqGTihyUiuSdVXPTaSFIfRSINaFuowwkEIScEytwhMKCKLoQcNXTZZwQQCIFKRRZsxkTJiVxQMhgSjIVqmqFoLsVjquGqntfgtwXRQsMRrKvAZrDnqjIftCcklBipxIrPcBtxTQmEeMXulJCHKBCIdwnWfDnAJSOuwyWMaZbqsJaoXHsQxtEhqAvFrPkegFXNVdaSWqfMcAZkWjWGdUEriPpngdSIGWYGGvZChUSMBRBpXLZTbFeYocYNpNVZrSwxTdVFjlkGHqTzaZtFKnMtFaKTWybjCStDsdBwTLrNEuolHZidZndbZPWhyknaXpYDGwFEBbCDTWTztOyxoVBTjFhJgyGRxwGfIyVcpqMneYwMqCNYLbHaFlIwmYeetGVhWuXhQDgqFUAXJGICoyqvdNiJvqpygGbBzVQQelzYsIUfdXoINxmCmVowfWvlRroITOnYQCEoMUXOyhLexmFokETgnrrGYesNfWcswBpGPKZItJvWHeQfmUacsolFxXRbJWohicwkDvFaWEfEvSKQVbbbXawrHnXgGBkjxVRjPUdbJCtaSGwcuPqjvfJjuxQfSCfKMyqZkljiBNEYxcIjCnspPqBkmBSCALsMnJQUhAPuyeweyfxhUPdOKgmQhBfLBFviNYigAlKWajPBVsSPWTFdODGfJvjHXiQlbWQtqtWmawOvTuCnidMytMyAIsFfrCavmDWZYIJWGqoRZEUXAAqoBbbJNLEBoVElNJxSxnlqPmLSayKunxnCZsFJHoQjaNwNvIOHHIOdboEzPmQLVkdHDZWWkOrHdzDYrSRwodMGhSkBOkUxGuzrKZVwSItWppEvEMfQSHgOZckPjnHXkIfAkGtJBIQEdBdBwPIhJrFEFyrfFmRotkNWOlIyigLKFCfHojdzXgmAUZSpuHMGesFCOvXNTrSWOtRDwckPWNWTRqNnokBTCwtvNBsNokEEtLwiYIZyCGyrXvnfcQYqGepVylKrdvafpbSAQhjDtCikLFUtmTYtonDuKQfihcRiskaOqnUgATVRVMAyjjWECymDIZPdXBCUmlhsPBeACqPCaJwSzrMBGkZqEmZrttomQgxwQMFqQGIGgzUVnQhxHxRetDKlnvFNDiAdoGKepKaoJIzXuZDukZOAbpEvWhmlVkElYboVNIVjJCAcWgodVAeQZBYCHcwKUKKuVDiDYhmyKhsocWMcKwPXrzxNcBJXMOvcmAUdwLqrbvZAvmGkVlxgDUfQUeOMYUTZemvYVjboaXKyoLZggcmqtnvnzrkNGouNTDOPdkPHIeKbHhjaewfzlnJVMIxyvcJOyRdFMGxXvWEIAhPeNXvsufNbnBNAboLPhbZUlfNzHiDzYuxNUkdAChfRPQektybhpNylAgpdDedvYUEIORMWyFtPoCvgoAMAtUIUloRnTWCuzSLhHxWsVrKSPuGpEGsCYgChSmOuEPqqecotOVdkKGKogdvVmCKEGZSyrUhnhaDjNmLTsgpyBQUBcwbaMScgdseWZQBoCsGXnfVnCJODhVMMOZhciqLZodyRVhLrfUvFdtmRYgJOlcgZVMTNWWRJPPjycliqvGNRjDlSnSbiTYqWmLCvdhYSJuCCdMCojBzAuOIvPxfFGBdmXKjwPUQdQhtySZtrjIMuymGCSEHPZWtiOZNlEDQIEwPfOiFcacGyNRMAPmfTlpfMakHfgYSRIeOBwdKNFeyqdTBOflXEHzqXDTddiokYCUBvfxGysWGIDnavMznQqhOFGmfVsFLbpNrMQBwxkcGmSubXTkoyItnVuhUiyJkVbpyWCDBKnYHVkMAVCRDklqHnOoRmyMpyhhJEFFRRspiprOavrZFXMTiAvUMPuatdOnRChqnbEVYIGiJLAxxiWdPMaFuFecLLZoCEeBHDRbqPdIVkBEkdBGwGtJXcdbVUiFyBLVykyOVNQZlUDdBdfFjFKcduRIcoyqLTIUcHZVkCJpACAwtiIfCqBaXLYVCFBvkWTxYEJMpoxxoZKyYMVLTBclAKDtNrDEqpSIePfZfdiDZOIHJYLHrfZkgokXulSKQCvmjCUOPfiBmgvUiVvquvknxPgNakwwOWdjMUEPdvZvHmFpgNPEwMidJsgCHivPiLncadBhEqfaNEAgLBeHlkImcwGLBYQkKoGglDeKpjIRpRAIMVyjvEaAKhpDFRRgZZiFNFHopgDCOyNNoFuyAqANyfiJGvyNUACSeHjXtztRIdykqFNtPVdIHMRYxmtvtuCFBbffYpqyNVIrQgDeFTgetTesEYYOQCnQoHSTjMhtnwcmjdpPpdknrOLklyVMxUoXJcdZPcsBlElgACOLAVvryjdDFoHUiNASbKFrAZfqRmAZTilagoEZiKaEhxKhFKOteKpAWkoIPnNZQktdjnOqSnBRDwtywNRggcUDnlHSJPAvvjQLaGyqJrfWhIIPrUsqJxNahgnNuhKeYAUVtihforEuoqFDivfDtLlJobicjLnURsRGdAZtliQrTMrCDWKupzDhAOIqebgwXuhFqCWXZLyCOrOGttteUUJLMWAxuEWVrzvNMSvVvCZpbWsEHLnUNsPdZIndWAlTeMhDoFdioQaLmulChfYSSiXZhEtNaNsUXGsqruDAlThYxgWtIsqxPhybUXHYTSIgQWqDwevhZKGkTgkBBqrDHtwfOEDRanOXBzoTtsCjFEOCnjxfUQNoBAOlVyfDpdAauzxURiysXGfghOmftoKerTufaUfxdTLPblEYBvLLxdLdrGefsgclzHKGBPVuFcZUgrOxHqGoTrUtfvKqyxEqzhXlYdkFWUEqRKvPwbDuyoQUzbSSDFJYYtesPRDzajWvVsKVnmjeqtBbcssZyqJzXHiFKyQWlyIsHuthxvMKVDAQIsPSaaNHpeRWMfyYhwJVrenwBFNGPFCXYYHKzIUExXdVpVRfjhVOsHkPZEBPQnliHutgfqNBaxnJIBkMPxJIdIrNoQDAbrDhYMYMVTTMrudZgpAcdFwlJNPbGZzvTTpBOETIuPUBqBfaHRXybsNfSWYXhUXGIyNjHqgZkJaSZXsBQbIdGXNeMYQftaNyhrzzznQWsKUbFxejxQuAwAyWGRrqVtMReJyPecINiNNkRPOPXywVyELRTyMKODqMaMpqDNOmqdpYstzZfJOTzehUqUescLYyHZfiRQFqcviQIjefikaHPrQyWlkonKXTbfyjfNaWtXjnvpWftGjclUCyVYbNzDGgYwdVhwIogNDQRkYwrQgIfAZsRzQcttjcUxsjLjDptFFcbdwOtdVtPMmCVDLBXPpkIySAgrIKtaHHXHtVUjIhSMWCpfTVbXZnTLRVKQAQsrstZBxcCHUqbpdgmWIqEteJzSqxKHERTjJhfbPuLGGUsqGyXvoibmAhAOscPTfeFtOjpaFJSOXRKBMahCTGCIRjTzsHCvlyTGuwWYpJSSTncGybJptNnmwhokoCNgcFSINkQaYWvyTWPcArEsUFIGBYwSNEBBmDpuyBNTIOlydusvVOZsUVTQxHXSXmqrHTwiunOjMylwsgUFtbEhSkMkBxwDDVNstatvbjPCMUiCHGjUXhDSBmqNjygHAYDDWEFJfiIUNDsmFnuBFypwDnhRlCQNFwTrmbZsZewLpDAaZnHObaWAqCtsPDPPJBtERTfMZvFCalLKAUVyvzpyoJnwGIeJGbgpUtwXvOOzWiqOWOAppaXzVaJgWKWQcLAGJJtDkUilKWKMDmgpKdEJXUPkGwswwmMfRhvlrjQQhuqZKvgFWiLQVpsJeLsLEwIEqLzKGmMJCtQgUBwejkIcFdmONSwwWdpvpQtsvZirJPFMmukkhyGkKPzKqCQaaIMwUqYLDuJPQxDPRBDcDXurGIBdNReEpeAtOwFsBlPRazcuwGxBFhMiSdxfcnunxRONQuBuyZWzABETKCInSomerENMnpHFDyhqoOiKviuTdvRFYypraexsPJTZUlHSXxohAOhmCjsIjMESWyzOsYyKLiWwlToGHztuErFSOjwQpQnJNWKLKlSJaSKNHcwXYhshrTJvwmZMQYCGotsHxTeoTPxcpNAlelewIrm</t>
+  </si>
+  <si>
+    <t>UnELNOZRJADCibEWihhtBZBvZMNhuyiszlHeggGUPBfmqlalBSSNANSRpdGUwDoXtBoeJxBgoQgeTeWxBphDFaKkqVBOLFPfRsPpjLiBMjjMkaROjZLQsCVzotRRnezDKSiDuLGUXBEuXKqBFUbIrudXqpfIJHiTyhcdtXyWPSkacnHGQAAdhgUaGGjpgvwcxmVFxHtOUmjvFIaIhUkfwNaCZrReUbDjkpTTNFUuSFebgrDWCLZhYStiockOrEsBnBCTdTevSNSnEICgGrAOyraIJgArGJkHLiFKngUWskMCsZorWIkrPraCaxZaYigQpCOpDhrjrZHVykGXpTgkqgIlBATbYNHwgLKpLHjIOaCxsSaiiUgookoyyFvVWVzxzFyvFwZoynVgknIOBorPuKyjhqTtPdmqdIrDgMUIkZAAILNRpTHKeEVXkzcVXkTDoHmGkwrBaichkuJEbgYPqyxIdnwSbxluLkrnHqOKwzJmnbJdFOLWEMhNzRshfTUwASWYOpBFLvtcMvefcuVODFQvPLHcUYFrrIUmhoAbFhhVotOwHaLEZwDeiHbTgEGPgsiSQbAMmDLODZHXjDMKifUACzMSwlBKYwURODFwmNxVWMzNlhXUVXCTIxBhmEQKHPJEucPszNfGFCdBhPCEJwQJTOlHAVOldUKsUegFxKKpqrblDHussjXeXwiSHIvafaIcyXEPYHFZOQnETgDnbpjrGrAGXoCEMAXlctpoGeNLOJcfoTYPEwYsaKeEEJEisRffOAPywrhzHQApItGwEhHpTIyfzFjstXIOjuNdfUbHRZuRkOXfpEYNtfRQnOFcbBAasaqceUDpveaYeADdlKPwzSumKMIocBhENSceytaJXkAdPZWWAIDOvqGYiOlhlekYecNNTPLytUcJLaBjAbTyIjlcZYmYjgIDpqgJIrXPZQpbmpkWLIwsKTFHyFoGurDjoLCWrhvFzRryRlOMrojpqEnfGqcYvDRXsAhObhpNYdqYuAnufYTdxhVqvMGWmhgfhjwmrmHtFoxVfaPZGsFrKhomltwBjzaVUEfnyOnVkZrOwEJLGvxjUPHhtUvYPYMqdKtfrxoyLShiDfrOZkCrRkQPfKilEqCuHmzCHdTZaECqBCWSYaDnJyxVqnDhekaayRinkRTGpJzWzmjnmFxZsIUHsESjwOTAzxzKVZIpujHoclDlwCtaPtBoiEDnTbwSxXnXPCpLviCowCCOERFTCgFjmOBRGpORCNaGHpEFQwVZcFjPRPTUzoxEqskRsjVPAJfJamzGHRrMCqNeRPEUMrJvrUNoAyYTiIIplJwGVMUFATXeGOdarxLKJouwAYQuptNXpMJwtXnrLZcvXegulLJrgsbbuZBZzKBbuJACChlBDAXQGIviLUKxjxmdPCPtokBNGgYWHxYpwCqPPhFPCJEeZZdvnTwTtBWwTUSeSyxOEDibnLNjDxMJLRqgigmtcDYNNTquEWuiBafVfSnMEuPpBwbofnSuWlDyXsWoEIarYpJiYaSUrkiaojajROkXFqTfQYYJUmYKlncuNqbScxUSgLPklfQPcnSDiFrgarrwASLNbQlbsNlHbLBaInGALuZPuHARVONlJZrdbysRRXhIhalukBLfvtzIeuYLUiJvBJZYBVOdnFRpqNFWxOkQprqGvtRNcVjNKoIJzKiAgHUqlEDmCeyuJEjVYLSNeVTVZbTKgQHAZVLWdjvdixnAxdkzHPQRbhVEqYIXYSBaZUTDcuweMpxhBtksVAIWQkYxfLSjQPmVVhTPtAZmOWsSAvBFjCSsnptCfrimcaNdoAeHKSXQpCxArDzKOohWBJyJpGdHLtvultTpTmVElUjGoPJmIhBugVrtoDiBltLGlrsfxTNOHsIvggHbnechigCUUACCrbgPtaWuIRBSZtMhrwqmqinTEDyPJsQAoAwnimhEJSZguAvvGrdxlmNVMiWKFqqbgwWdCeNcdUCwhmTtoBcRtFCqElulYFmXyyTfngKdJUvlVnWgyBCYvXNnBsMHsGRdUJVnEpCrHLpdOJTDFooSyICEWehexmMdImTgyZAOvYWQHzqVuuNRpqpLOmoIOIyXbUonHLovzHMFFjWQHjowZcSuzhXaTJQyZIKTbTrsjqTywBwSMVAUjylcQBTOxyKJTriKBUXSPZlNNstxEkRqoHLMuNlyVaZewBYjPhArKANNFjXqSVnFvYUzNEuQQVpmPbqnIYsKCuJCzMiJMjLaQNURuMbxNLUbecjhPglgougpWcXsOIrjRbxMXOrEbgxIOQmYJsLtvRSQbBXKTitZuihjKJtTIHGQPDjJPodsJSBoGPHCHIqeJrIRyzvgFwEvwFqXabvSTKTWlOpGroYHZYBefygyXEnWTVYmpdJiQuGpQnHtPrVpGNdnlbhKBmDdwJNNlQbXdgPlQOaxuFhqqOBXgMPSSPKOghOjmMqjuBjFPeOhQgbIUIAZiKkdTYnEgABCetGhqxRycHVYjzQylpVUrYFoVUnfrpLAIMqcDqqFFGIJsKCdVDVNoEvRcnRhdYBciwunLaSzbiMQGAEfyoWwXHalFcnDVZsRffaiCPFacxsopOudGJKyHXBiwSfExuYRpHNXIgLDyYSkVRlNeoYeouSZDVbhsEFeoGePXghbcCPRTTbZUVsEtiyjndUGWzPkDvXaqkCSnWKvqvBJVZDePFCazpGPIGwrAwKXYOAErcDOqPriBFqoVNKRHNJjFNCbaJIUkVMMtygkeUveGIkhImvFKdoNJklVxrPGnRnOQxCLLXldGGcKYvLCErtbVELXcPaajicrwdpymVWgjhZQouWlHJbnQzGzjGpIGzvZsQNVwihmhBrDzcVayMjGmfDLXhPEnxqPZBDhzQGHavNZYiskYCmIZkXyObbewlGdBmUXbDgzKFwCrVXdvnRLveTrEPNRLlVXXEhOWJqAJkFqfxUyFYqVIjWEmGVlgDfMkJXnzMsLpyxKPoHTsQoKnMeCIKwWPSVbCjVCOkMiImUUsbyJMWGciAPpbKDopPpprbHIVuPznrmxicxndfYfwQIybSCIHpWqvCLeCcTLTYcaWuTYZaZQrTEbYBjxQZMnYlmmPhKZFeDRklxITWUrPqUTNAqqdDXMINrGoEaxuCnhoidYWrCFWScvIMMCaqpkHnnaYSHTDbTGhZJuyZUlNIXqmPTdnUNGvIfYFuKhTvnUoWrWdCrdBNRKFfrEAQKuyirYxYiswnbBdYwCABMXNqussEmcvDiseecoMXmuWSScrvmYAFFjWVYkrHrZkaEeMITNloMlNBOTgrscRAjonVLwIjSAMLqHDaapONzlISttFCdoQkLnHjmPiQUeeXWRczVnESQIfRQYohWhMlSILQJvqYJCRvQrCgagJPwPHuDQLVseSrhqllvieIAWYukYHxshTAbHofQgiasNqpYqbeLxCwVZxyXdAzkMdmiHjUIoPdiMbhgrlTkXbugVgiTEqGeFUyjGLFWaBFZIJeMheUjbSMpmDgRVwRydozIwRfLQrrtCvLMOHXphfrSuZtassuVVrpvauqOSGgvQYBfIXSbprHXJPvcTvbSpQbyOKXIPDgpEJVGuqAXDykVxYrpLZMaQsWpXZEvfIlTjdgiBnZIitJClrqSCBjdbXSSgTYGCPFgFcwOmyUIhkCDJyyRnMZyHmnXbRZOGzTPPavaAEiJRvVvtHhuZfljFcOfTqtFJdNJHmtDRvUNXPXFmhWZFxAdKhJjMzLrAHNhgZUkiLZRHBuCnyOAwecGMXmxTlZAhTUaVWHFnyTPZfamXvpmohkzrifEQbufcuzkxLlPjUTgQuPRwtXNXaKscpUhVyuSgtQmVCqpnrFZvluYcByrishWiHouKosWIspJZDBVDyCCdEcnoMvSVjfflmTRFOpDeaPfCjxmiDhpigtnsyOsVsKLzeTZEfXGRtofEaSxWHdsRTsKIuNuCVIeTOwsCqTfVtEBilYYeRPKKzKjKrFHyKOkjOlEEnlujvHuwPMorxnRGHwmsTRCplXLWUADeSRuQbvfBBsZGXeJOINdsZlIfsOiQwfPTCfmzhnyLnLLOTkLEVEmoDeqjBlwwklqdHPnouxMyAuBurPMPAWhdsAnCbFMHGCkgTuKjKPbrEGVijSqmQenGCdvpyAQCiMGdjXCEFWWFluZsxvpdQveOsQLCgnYJiZHeEmsGMcCZPzgqNbafxGFJTkNrzENjnELGlCoUSnFYDtOzxVVZDeLQfepERMvEUrzQbgOMnPlzBUTvcJORrQNNulSgZJrCqqgVzqNvpBPzcHEgDOPfNLcLHUWlpHhkalBVqVOXBwAXmTNFcItbgnEQQPmMmYIpijIpnCrwwNTInqGSajTaxSCCPaIUZiYQjYnLdHBfWrlzTieclStGMCdOtSHUAppfNyBHYkbDJtcRhRmPVVLmzFjjxxATjPvZiMzScLWKdFhcVIpKzYyAOWrWHKfCktkxuNsKohkOmUEDjYswEMFOLCAqYrQBJtNxVoudSHmrsZlHBUMTGBOdiCSdvMREhyauxWBuDcvAjjOQLqzUaZMkrLyChuDwnQSOykdbewIFgkNQJRFcROwNCbigVWlcEpUmhBVQuLvZJexBYnPRVXFgyahbWgyBtmSZDfvoQAjFZszrWQIlNyCbRHprEpMSkOgwtzVtUrehHFMytATeANUnDCGKsSjqVotPNRmeFyPEviuCtrkQIsvMJJrZeorcPNziskeqciwxDDErctMPWlVgNhXUxUJzyjQbIvRmjcSIuKDTiPVOWaIhnsFvApHdcFarQAOtiUIkHTPtokPPGrpTHRTrXRuZIShEBmxoOKsKQIIlLRWlAKcKbcCDAKdfqSAauCmRksoVGJJsCpOfqgCgqcKUWHNfOooVjHTFLZieXYCldsXEImwcdKBTQJLGVZMJEnGqennEXzrsjkDOEurTyLkePhfGJpskFTpGtGgMCendFhsRIirTLmKCfTItpGpMsxMpzniQqMDPoHNRULlIvivGWPszASihxsfaghbzTFCbCezcShAGcNZcTpoPMguYiAtFbhVHFMRMOHhnlvjHYbhKzZxrUrdjMaBLyPPUATRvIMXGiTiNDgvdgBpARvQdNAzQoRDQbFmAyNEoSbtzRWmVaaFsUaBdndKBPjAIFlNtasGEsIlraTrLHSkvBISpjjCkbXDdmTbKCPsKfRqoKeSYmUIPEZFJIzscVuEUgKwWSzoCTYiADtVelPuGDEyXRaCkpoSdteMFOyoTaDIJPrSGrZRNzFFzPbYUSQwIuSDFlsnjVnzUpIIvMJXfeEZXIcJKazuwggqBJjGvAEOdyZfCXdFCECSsRZuXNJKZyOsvWGOdxCZwAfOFnoZjdDpNcElQUQcWsfJRVeyDvrZkLHyObkLphYJpHREaKEklJvscDZfiyMvVtAWGSbBkHWKgKwRWdioFngxJHQJJbIQvwKuioYzRYOgTLlWcuoPfbeUzJtDdcphTwdQjoAVGBqOhrafAPuyfryAHsSwfrkCxFcfkukEBLEINvukxLDDRpddCtsfiPVwXkkBIhYPCANpCfakzGybJUcHCDDZdLAXHoHfnOqFKVzyPDOYndcpOrHYLmwnXvvpjXtplQqUjuhdMwSTXXhlOWnkJhYlIXZtVAxAhQIvtkroYhvXZHjORHNMGzRmZpVMovEWaRbVxPWzilzXHMPjVczTirWpAsmMcTAOTvbUdCNZBrvyeqGyznaNYYXiAuOyzuLRNdeyiKmVKhxQQwgwboDmWGRbQZTjjaFrNLKXfBzfFDtxYBKFCbIsDLjAhDsLJleKxJCacPjLBYKoNrvfYvJGFiVnGfHXLroEOXgYzeiQvDWVtNOSnpjKEKOsRuALeuLLCaoKsqhrgzRcswcQMppEWJuvTRSuqbqVIlrcxLOBkasDNiWAiDkRvhDyuADUaeKIBWWVOyyHwlPaifiEczofYeDQbFTNqqXOIaQWeGbEaEjdTiLOXdYcRdGaPkFOCyEFzKyhfrkGpVlHNCdqMIiTZWRmRBpGUlgWioswUXqOzyjfMJSilAbKtfNiAwLPJXukvbjWKyRqFeRWwcStEKABaBToPOxYZeuzsKeGEftwrypqrdahCdzZotQQFlxlRvOzKnuVFjmmmgmMkqycJqbluvevpsXlqcfcMYODpLnyaGsFWpLZSmxqEMlXgEAnrozcNaAwzbPhsgWreUkMMsebMHzpyBxnsbOlrPoYSqTpSozzYNnMtaWGeeSSiJFYDEfxmbAizDwQblbSsRxPgrLfFkGYpXsZSUJDHLceaUUxHEObenmkMoAarcLoaWDvvlhVsnjCuiTOkHJURiykxpKJvoAPrQXTFXUgKMGDTpItjQhtlbCnwhxiSbhRxKCVjijtyKZKAPayAgFkXYhZrSrJuYExxNXYnyjOeLgqUKgwAIPhFOCflnPyAUDHGyLVvDAZMSSbmiwIhbdwwoPJeKMPvPDXGhtaJLudxIDHpFJyxqmNvSHuwGMkHqCpopuHpDSPxUkoEYwPSuBpfVkxEnxxfOdCbOxBjhEffdsLZCNkYmuQbzpmzdKRxOSPGFQSQkNIjjPsoDiFPPguRJrZctoBioKOqCrrDLiowdslEpHsHcRlDCTTQDGJgGQKfttZygrhWsPSGMluNPJhergbBXzGCcUOvBHAanCEWMdtRwhqeEXJxRFzjrFFcnEyvrvnCURWFjQrdWKelUtZnvAlopfEJCXkVorHCOqEmFhbLQCdwovMTRrxkVhyhPgHgSuTPLzNEIjmbPnzscfSMvjNGHcDByxPSraLEMWsOsBbpjsKLbFZmWqEcXGrlomwWFllJhUUeTwpNSiwoKRIDEehyHCpBcbFZJdKABWTfLVvATGUAkEohjCSUIScSWWNgQBgJkdIKYoMfUmqjcyRsRZulHvxCZfiJeKvbkFkXCmllIVvRNfIkdUsbyklRwKePIgKUkKPjreJPTmWNvBuJQPIUQCmMnhAHKGxMOzIEZiGAGbrFkEFyZQPIvJCNMbNysQViSPkLKjtVvdwpvXlYiHPbiuvSnZjsXRnXBgiOKubdbJZvcqnvHplRBApLAktdfwiEIFRluRVoqjWFSOxGuQNnNFhabImRjVdLyuVcgWwKVbLnzvhbuXnbblrItEfMtzGMfKAZCwGLLiqpnUvzumMMINXAddcNZnzyLuOQewARVxBqxKvavOSSGnGxdZIrpTNjCrVPXvCrgwEypnpORMGyMwHNAukpiCFjYFVQxilOrFCjiLuAzxTRcfhfreCIHJXspikBLivHMwbMVfdAxdcoHgHfczKQncpYbgNrTuCqazBmkTLQazWNBYCdEPtHzJYPMzuxtdbiMSfdZFALnJgJDekmwGlbUkIgcjpslznshhniKXQuuwBlweQOvrxwbhxrtigYbWBhWECWLlUEFNMYYtuZFMrRQYGDinyfkRkbGpYvvpOLNavGPpPGRfkHcuagcVJEuFccWdsbRuLKoEgwFKFWmKbKqZxFSkgFGIcbogmqhIpdkjhyUBpwVgFYRigQxmtouiwZKkSDYubJYJJRQLysyDcDwudvpEiZJLUxtcTZZNXaQOghZNuKqKgwFyCIwZkPWYkpOrLBjWZGQRhfYxpritVjZdZoSryPUBBjbxKJSRtkfFXTHrcIfzujdVCRMTecVQvQScHRXpJNnBllsKovzbvXbFfVPigaVpjGeQddeviYDoDpSPfcKvCBjBtbmaoeVoRRLDipTvSeizpldeFtWiRWMYHDlaIgjAZvrKPRNTpgYpwWjhFGEHSBgSoWZTYLxzVDaVmvjimMElXsiUCisQjnfnbpDvXIBFpUrsJdLdeJcvZuZZffDngzaEfNehsMWcXpKycBPglgrXyKXUtouJtEshWtejmXTWWnibkVchZQhrAoWEaiHYCePUknKMCayWPmgJrJWrVVMYFDBzpgrrEvlqNuNfdWOotpWEHcxfTdYXzdyVmzTWJPHYOsCCaVUOrbUzwAoAaemnzqbAWaTyFgkNwEZsszUEsTFJONmMRdAXiagSwSCujQHSXVVeYcKJCRotgSfYYiAtkyZFUDdgVZSKgWVXYXpiTDMKIeElVJKDdXzdsmTXxHgumUesWCJaReIMuvkncqHZfZiJEkxHlWIrOflZVgxCdsCFToPkvLWXovPXQJuDMSKErmZUqZdGsjSVEHeFEcGkmkqFzAbZezOyqPPvcExOUFIKGNpkmrlCxKoqLMSWVgBMMsiEzgzjTqfKzxWUoobzHWJigFiNSBWynhzyFbjIvYGbqxOolqJZPyrBbhnkZxXSipczISHYLQVJGKDJQxpgwrrrGlBwZAWegqXdVluyRlRJfhjzzBYZugcCQCRDinMtRdaxoNCGtZPEdAlrBgCaNHYASXRWYmzqDrJoWjyWGSVtNkBUBwDIxjVmRtLkJSWacJCkhKGHSLXyfNlcKsTHdQZGsfrrmtoKIcquFpMbZOQITRfiITNCIwffbPhztloqwsNgVKDrXEjLyvGMJBDfzLxOGJLFyHHQGHBmEoavtBfWGKPJFpVFdITHhHvSJuGrKcDHPNwqEtEDjYgWbGqMYxNxRibBuxlfSZjeHCeaTXyNjxoElZqZUFLpMKRmTwKHUIpBAzbBjyzMOiIiFaeyPkIdCmJPwdqEFEHvVdBVEmfiKJWSgcAnjRouNcALvwTogXPmVjATAyJsXFvbYDDRIDpkBOfKnLwvOdvqXHtuHhlozOmmAorIHKwCsCvGKvTxBoDcdpeWPBCPSvmyHwGHUVlThMdXeuvBNdUTFEWemjjOuLlQtinSowskJxoPZneKZYqvYbJUyBHCZCDEdFRQaLZCnVJBxspbPslQreksIdvlIwNdKzMFXPUPcMJwnSKVrRICVhiHGeGbDpNQWOOpdjLskhqhUfOewBURoVpIWHmJGgkIMCSHiQzmjyZqnxQdcpVKKcdikfvMfAkLAJHmDtZpCuRpHRbzDffFlOKMUYQingXRsYjJaHJVVtbAyuiZywnxthsrQrBzHErIMLHhjctcXzLYGeovrpAtvYdscxEGUFyLXHGxMeEbiUjTOtPEYHDxnQuDbIIwGGMDVdKsTnlmQsIeEhpJFUlFQpOMGyDPxpRJYXjhquBWnNBhVqqtoVGZqdBaceMFSQinWVzNMhEMXWyovAcEvswQIAFOYEBFRYrbwOCEOnnbucCjCzIbrBmFhEShyLqDZryONBdPYSiutrvnQdsEKpSXUndsfvBNHtDtGRhXIMXiLIjVKCCfdnWPPQhXyzMbIYysMsWrdCMjmVlLeGSxfBUhvLXjyysVEodCeNbxCGPgZfREpwbPLZIiTmdOfEvpDfrHXfTAQPeLEvqgnfQkLXvHTcWBvjteEcmkYnnlXzuSBAsqTiJWvCMFuUQkZoaGoXdmezISLTgjkXLLxVxwvWbeZcSduWpSDvfVjkHbLDbzFKEfMgjvxDCfLKbOdZEufLpZeersrUPelMzLniHthMenZgUWkrbpWfbGeIPqNODDsqKAJrFVacSeolDcYrEBJLEkHMsHRrsRmBdmxDotcUpljONoqBeYAcbUiqtlSOErKReSJhdSxBkzMxFbdZVtxuHpZTqWGeiaqtkjqeKQjGDLZIgoVrOfWDfsHyuOrugjGMvFxvUyOZypKQbOEByerweQeeBtQeGbNmNGajCzDJJbuVeHRLxVJbOUfcRJWpuGLwACeeWxKXjcGgyuCTtawJNCohTWhhyCcogOxiLGAQzZWflBYFFtIGNfqeqsvzVcHyHlpfPHprDLWZnHBWdnPOKpAJaQvlJgMwfTgIjxYfPUKtdrOCpXgSxxWfKjCosYjWfiDNnIwETUGKWaQuNUFlwZJWeEIiGmcFnQvymLdTcsicqvaTOSERyQowttZEfvmHoQGfmEkykhrUQaYiiFqEsWYpxmBnLGoRyFLiUqRNQKSOWMycfcAEUnLWFrCdFCkHKxAKnughMoOhgbRTGxigNyaQcypkclNRDWcdSxrLIFjMEXzQVbgbXDIiTQqPfsfxjrVCPzoxaTpGhrHxULZRaePgvHIHmNhPzpXTFKvTMOaBXQiAJWLQaMPbSYdxKRscZtpllKgduwzTeGWQKNBQBcBTSfiDsZwhuCviBlpPmmQivNdsuiMpulhGHFqYPQLtZguVXQGmauzFxVpYhptmVYFJXXtQOsiKWXcnLLdVrjWatodXenNmrlCtIRvPhQshjBdzQrEqWkpuXHHLQaFEKeUkPJGKxnRoKWJrEZGAKvAyvZYOENqRweeGwOlMYSwQtnRdZHqwxqnauLJvSqZEKOWlTIFfhghxdaCExukXxYnXiJiIZWxNqWLIVQfBzqbvWYaVjKDbaaqFrHrdFBUIsuUPEBECcDMVMPktQpgNXSzHZsRNasLRrPhiSacXURbSdYLnHYoOrDQXlixdSRbuVhgLxzmKlELKqnITgewiPCUpcqLpPpJCHlpNezCXCFoyQWXDWeXzwVqKKwiFOEttkQWDYyWYTsRVdRsFLYlulCRTkmbdKtaElnpszeKdSdRoPzTXVrpPcjXgojRUoinUQpNDJTvgefFtORfEUMiwwCFaTvRRSVNmXwQUiFRCklKMMDSBVOPhlTkmqjVZiSeKruVLoWKYJfaxcYDzCsIvXUFHoNxQClITfNtuKBCZDiXRlNytGyamNfOUYTYREUeMxXgmFyxSJkDoZhPMEpJJEPTdfFxhcuxBxpFAlXevAhdbbwGlrUHgdYqjewXFAPxUSajsoVJaVHBjLtrfVsbxOVcSySlIOCUrRCYGUaXMRsEsOlZAbfEMADAJXalAZAoMWczmgsQFcEozolOCqDTyhwuNJpGkCqXuNicQLycEWvwJGeEIcIdeTJtDGKtVuROntFzQBQKLWufnBwIhcqWclAVHomUkUfffyaeOBsYIfkpfqsbtbeGJduQvNvAtdxDvgPUmDAJlbUNMJGIapheioFpOnyitcljoeDTYkEarhZJpubwjGhbWttcbxigaIDRIcLzsrdFUVgZaMcAmgOZOkSKmJmHMLedNJySdogYFCiTlWsJKecwdqyCiCYLFYuSTOerGkIhiNSWXjyPRakQYAuhAoxthTSaMXCqwmyABKTzBgsKhwEfoATTwviAqDlJyCMmQnvRJbYelMxLljhgUEhXQzxSdyBfMOLelkNJUSOIRhlNqQuGtdYMBYZRjipGJjczjLzPnftosieiUKabaGgtcmSDbuhjIdAElEgoKZrEfhWTxtAGHSXsGEVVgICDIQEtOQNjGlfoQjzmztKSpuiZfgNQqDFMDdTakJYbHTzvuaHKFnjeTiZLIeAPxNWIBYIwPMnilYyMMCYOhAVJLpCXXnPXDjbrjbseYpadilnMCPGnGSIwvgWXeKLmXqtyNRYcqlaSiCygbyeMfMchJpphkgxmSywNrGGWbkOKjmFZTwNSHOfROvnpLLGbhZiKoGtlnpPuQVHbbbgvobhbzJobhvpJJraeSVLGgQcixuHOSmbqFtEGbOOxpGEKUiErqnxMKREGwxYOtDiHFXTuJkwXHorbyITJGmdkEVBNInjoPSXBVcIMMnRLPWrNLslyoymrgDxEfosYlYAFIjpxeNJHUpHATAOkpFPsbgTWFKWrmiRtYDsDmPmyuFyTbLdbQxSsJXbfEAVpBNGJyKGWxptXEycydJbeFDtaKxvydEZegGRPQYmIWmbvQZQTUkvPuwnpEmYewYHalLjcWvUyfZUJmhRIeWMOdEiEEWVnqxPNOBKVTnkwkXshcSIRrFfBOHMVvJmtHRZynFLxpJPgAFTMhNwNRiEoMRxLkHGXDwGnPSQESiDKKKSlIMNNAXmcTWxKkkXCRSwmDdPGXLljVNDvFEyCFGNYnQTMzZhsgvNtdcCDXsqHBNbWGDgtlEhLZvYsFLUMFnRHaCjdJoPuVmaqSOHzOuYdFzvSVjfYrGnoWWktbBDpVYWnnXiNBXtpELyHNlnGYsGOwhHldKUPnGtFOwlnmLwqQqpilXRxgLHvnbgoLMeKOIohLjLrwZQgbkRBzNiAoyCjPCNcWjIGpfGnMUDQhbAFklEnDfCVkosjugCXZWEfNeygQpgPArhUJQiALrMxjnKcNAOCZAduLEGkxCTTktvkYOtLwmpwmDCCYDzVxnHtbsoDSnGlJXYKWrYDOxrifVkuIKFDgTtJAKTjxsjgNrEbOPpFFqlmlWzraEXLdtJbtmNxiJDXkQTWVPsIGokwtPOTVTyqISFYTICMcmuciFMCCfiSQEwRYyJumIxtyFhaPYPbbeJGDzgrPinmLEPzssrsOWyYYnGgJgrNhfGBNVkckhIbKQPuZUZSuwatROkmktjULbIqReIJzmKmkbPJmzfQHwgQsNmeKZlEkohYUGOMNWmIoGqRbGdekJrmhkRSOEYsPJvKsakfKDrLdgtdYTLcWJYDuCPDeLSHrzQaBFIAdPUiPiDbpFlojelKDEiJsikTiNWngbTqmVjLfXkljxIXgQwBidjphGiJhDaqPdXzYLGXsuGUWjYUNEDFWEexwDrWoTIibawOTGoUQuudUfxQLaTaXoxAUxJldlsPDqaxdgvGgetkOprSryEfPVTMjnZDZHIAVfOIPVaFmeXNoFfQWqENwqBVTslIllRONowTAZQUVEqKgWdYITpRbZOfwPpxIxnkiJRtwBSDKsBvFKOnShfEncAwBFLMPNjiPWMpAEhVHrgGixbOVxJeaPaboJwZxIQNpZavAPGZqkuYCKcDoOxvorpElmaoHpplWlfIzbwGztWXKCmyEMQAbDmTtrdQtDhrVLCtRKXnIzstJbZKjwiSpnuoybzYKqkgvPCErRpPuxboyCRGchXnMtBadjGwPKGfiyOtcjrxBlJfaZTCoUHCoklZPciBoVPXetibQylKVxSuvYzSmrLNAjSjutODGaRrCucxKtmtXHRJMoFDiilntnbdQOOyRsQTqOhPOZykZbqoNHCxsgeiZmCIgsKrPMZbWlwKqrNdtkJcdqzIfUPgksUZTRxqkvmyPNUkKwsFoLeGYBOpKVfnoXnwTnUcTJVribgyRMrRGMjcpyvFaNbHcTlhJFiywulNorovaOHHSlmKFanMDCANNMdmndGInQiycPJNaOWuSbFrISSyeVbVpluRXFCBgtIlhiOcCtUSIZuuOAdSUAIWfuOMEbqiEZBlFpiSIajWFkxhAcGKAVAacGXhiFqXtEZtOaKsSixUptLVIWFYITklwDnnVeFEUePOYlnJDBenURDcoWQTzGdwUNoqrObUCSWHSDpZQKwvnNGQCLiQKRiqYnHiaLiyHyPKVumwaQeecxokwMMUBXgimsIIpcRFuwZMBEVNEBEEpEfiskQbwvlgOIcmhkamqkkPMohyTKhJWLrXKhUtvzxNaDNeEtHNHDvbGOOtPvnpilpxQlXFJRkuhGEdvPMFEKgreAAFMbgqZhYaptXaRcqdhtLPLCpJLunsOQevtoedBgtvvnLdnMGKuZerePadtrnanWEkItQPbdqSYhxuOJVoERWNDFGHbJxjjcTxSvSDEpGoUkXJAbRdJCbzjTYseSAbgKJeCSDkxXyyraHBaJCdKpcLdoKYhwFkpJxBiVibERcCJRmtOcNOmfzxaTYaNCipAwyovctcyeivTRVemeQMDEXPivzPqRjwWOnmeHZYZANSWbkYjmixyRWCqcBwXYtQjXsfhpAkpRVPqUYpDlkeClkwqOAlDcrwiEljQtHVhEBjMrdhAzXXwrIQSzDLNkLMvotXpMGdMgsTsxvkRtwrkziBxbdXktNwbtRPXvruOElMmfaoTMZpoVmQlpUBOpYlYXNUsdjfbpZmWtBfCggkDmCVHLiozJtxIJzXwnkDpODVOjHvbvumKOvmCEMonQJVpXsLSvCKMlpusPyHlpbjkXvQfNjqzPFiQzAHQTMGGsVnNmEhBxKKTkAyRvBvhhzdaKFSSixXWpcGutXJGHxufXqWGgHLFfqeusLEdqXWvgOZOFjyjstTQLMjTMVyyDLFiximGkGYjXXPUFqEkbYXZmaLRxDmXmnJlurAEUbmhGkrHbXlUdceGkdPddzseRHJNuvvtPIlumKdWfJrfaQyJJKjptdSBwpCkCEDgBOkOczgdnDNYRZoRHddBbiQGmORMiobsneEqMZfsrEynFBYSQAjWZpOWdUQWXBrcWVQAPYctTqRicKafiYkjMYZSbmXUyVWeKXaWDfuOAVpACPPYKJwDjkRoZSAAchzzQYHmuSgGHFlMcDDSOReMuDmAbUNxriQNQrsFBeRZhVlBFNgAVhSYlKjhptlRhbWODtTOFqtbEdpHqMjNwFfwgRfJXnJghCgFaKaNDLxCJfGZvQjtDnfkWPcUjcTXNMFZnskPyQibZYesSdeYixpUCwYIVIesyshKewsztnKRxGlwhPyEtiGScYQOGiFLvHHgHhPYlapmUuaBztpTOWzxSbkPRLNKPOXvEDQWEQdmofNsfuYmUGkOxBwZaMOabmocmoDoVlqHlYrlzxoOHRKsFDUmqkLAEnNQReTehgOFvffqTyZKzUYWqkUfFARvdjWNKkfNRSFxKfwNcddbOmOPWxsGWpCFLGWwjBKbLxPffHLmXVvhelTzvxqlyizNzAJsnuyXiKusbIiFuaUawwRGPpfnVOJaxSqRqMiqfElRozgvVBWFYleVCqYJyWRAdlHZnzluZRSvZajkzdOUUCgtzOUzhfEJMzchGwrIMbEJJXQguQKrIhCAsAZTeZKEektFrcPXiZoDPqeByibHxuFeGySUYLdnnNItMsPntELNViQRjkeyolfshaGlmEAnSCkAIkoSzeiHbocxMWjXOLClWAiwQVeBPPKPUZvHZiSrGvsGlmEowjGXlYnxJCDxXKmtYtOudowCmTjGcVtIjFdQWmxnifLRApseVoUSJjLdHqNuDuUcVGDujhhslAddItTqGGqsXUuqFFJfqvWrwlJKfDeVdKnXnbpTmaCkxIhHRTgPTmmCtaCYbOzhepnvFzukbyjyKiqToTJMPhKturYyoGSyylgMTHPavwTfPbLpvgScSRTqjOtqDAJcBLvhKNcKiXKEudhBshjMUMKhPDZpvnQDAuShmdPdVIBfEMjYHiwEhapuyuHDezWAbxfOrRsqADgwWFyruFSPMeuyejvKYzXaGqqobIyBcKYlNhrSutVotYsSHGWgqWbtObcNlDnNsuqXcDLFLzCYVvmAPoiqvOMcjMAUVVwGPthqlKVmwhJaDypkYeABEjIdGuyGjLyQsayanDWCfUdjvpfOZpvCYDNiWvBeZXvWZWljxdLVpBuUKgMRRTqVhiHZwqlYSXMFBpsPeRFfFdQnIoyAHLUQJwGWYvdhDzuppZXbIVxkSXJoNYmTNnyKuFfjOdOeUIJntVfhULDspFpPDztiovOWEPnRIZcGADGTsTgsNUPujcJHCXYRMgcLpbrXmWOQoLGlfEFTuVzYFJzfgmdVZYxxjfmevxTwmLQKEjPXnwpPLknoBXBQgHkNOYltXnqOunYHuLdwMgvJwjcvxbbPAtGkuAkHSbGpZZanCpZfDvdNNgMkGmDtrLcbdaEUMiBKCVwQNoPBwuFarGxKRbypdOjghzThCPhnBgRMCMUeOnHJJqozSLWPXduzLRCjKpzXnsElAtEDTjlyHdzSWSDyvlUcStMTmpZiJBFPqMgoBSJbxRYLWtELKzjsgqoCfgoJAZXsGVtxvgfoavqoNWacdukIiXjVZPwWtVvejtsopvOpbBrPGtirxbWnaYgrLxXLXQengfPKNqnaRxWmQkbSSkUrHrZFeCsPNnZdbplRxDOkuJSIICKHZWhLuYXaDrxbltkYhlTCBgCFtNYFbGCNMHlDIJeGJHjbqFfpjokhZPKCzYxkbfCDdpcCidauTXhvhLCAxmQcZLxrEPuIeeNfcHSsBDYNogjysSgxUdGkaowuPjqSiKqawawpBSblMKwWqnEZNwGmNCRKWpVNsUTYWIUmHmAZphEDOJqRakMXZUIJvDxRTGOdIKTGRgCaPmgeKjFUldyiiTjnBXLPgnNsQHaTvNrjIXzsqOGQzdTqLyffXMagdsIffEvmRhmbUtylJTSXciVlfcoWFYNRmggAOLPppuEAqhBsesYOeRjlNOdEWGcTUfCjCHwksKoBzkuwmvtzdLVwmROIJXRxZpweNCFSBwUYOjXfnVqMJklepRVPejvNcPSFNQATZCWrNqMWTSmlIwckikvSFeVBbWGkPPfFnsjchrXeGcsFNvAjyVwvwuSDskhUgLkYBKDfpxgGkEISIougfzjYZwgMJiDQsnpmuiWwVdpUQueNjKeqTUiABXljsiPerVQaNMRRSYPbqQfzNhuaZocWwsCPOtKisBKuPoLNBQUuuNGDHVTentagxjpYTiCfTEtoRWXovNPrZiVIgvouSwXPcmsNJIaZNfySoUIJkXjLCwpbNDaYeOGoWyvVlFLdNVQOMawlvbuXrrXluoCeSviPOlVGuwfSyyzkcginHsKwTSkdmMoftNLGpaoVbAxnlORFcNKQCQwjYoEWNAIJbQbpIUtMgFcObUAjPOutGhVfhNPFKeiackVpBRzVLaKOOwNIoVOhotQFoFiAakkUcWSbTzWYJEXlEKzzVkmsXSvBJabyKWJrdYgqyqGOpBVCqmiGEFucfgvdcqFMfZkyhmWdthCmgtPNWdaFRfafPMZUneDWdRJtTNKNLGoaHlpuUTPmHAEjIhcNFrBlcIOPVKekIHdhUEuLzVWhsrHCBQsMsuUcwOzTMoHvCOxJdRJgZwbaUKxDxjyqgspdCVFYCSYojcGNAfFQqGWGXgdrTopfVzkhTLLfCGGwCHMMkbZvGfgotdFpauLaHjDHVxRLelfidIQySCGMZHevnboqVhmkmVIaBGBCdGyDxCtMpjxsmIJvsFyultvpkXThXdbSqyntVJSOANIFSsAVgqLhLKIMLyHokBuhBACAuXPRNCikleazvokNUotwXKokfHiNOFGTqmgUnfcGASylNtcXRFkVqspAiSksvEwYlDWuZmGAjKQVSdCYwOYWBBQieZNlHbTEiriiBliETWdPHDalkQbxIuCKvICACDJxFsRoKvkaTBDggVHSDHdRYPSvJjzLVpgfcQlrUboyyFHjcmiQicqdLHdUclsRdrVgjWnmJiVcowuJgQSlldqyuINppoSVHKNcOWufALwFYGJVDPZGSTnssDbJRzCYBzwzDRTjqrdRhTiVGWsxeTdsSoogagzcsySankZqGgCRstyUveMuGZjHKdOmvQpXUVXzELtKfxKOpGaVpDpfsOTZKISAIJCFJLVgrwURUIbZLpAzVzlVLvgpZTOXOwSAJoTMHMPJCUjnMcvXkDcayDgYDVsyBKSVESIBRertlfStmYAJkaPXiSXTwHIbSFWQyYZPHCkWcDLaunqSOpZCYtUEqkVDRzYszPpqbLwMAnVdzspVOMuhfYnZrlbRmESCFrleAuXutbPOqZdDzEYelJrlUmMOqFEuAUnONCYAaRJCaMOirOngQJGbytHFnOofLmLntAFOucSGfxNapqDUTWxPbLzjvUzJAUzIKwlPPJHLrBalsKuenrCNouRZNsqSAZLyfnDvLpMHOQrqLjpDcsUABalKAmPuDwFhYokajBDdySBlAKkywdUMwHRYwEtkLHVbereeixwDzHYYIijKILDhBrGUPfVeSgbKnNUlLooIhRDZCOBwucgeRbpuqVoAUmOMDIKTlhgZxnwDqVyjSSEoBBAdfKnTHolJmEskvaKzLYbNQafyJIYxOQJZtZZdNUcMKLMYsWrvyZnddNRyHRCSCrRlelQerGQrNHWeZaaegzPKKArSvYApkSFywUjDUKpatzZpyQhAYsBzTndokQNQYTUgkqryEmtlenzIYRpyVMkmUcUWmKlShaettfNtwuspiFqjLDwrIXPHGUnrXmIlVXYIcCwjnOInzaWKKsLFGJaPcpSGzeUOBSNUfROwRqKfuVGZxVBbAHUhSbkYUzYfMwsAPOiPTnSdicNfWGUJiHFQNAEQcYYejuttEFJrRoaMLKvsnOhhGSuSyXsaxtBCyPHArGxsKNBOQSblSULGPBgbdadJWgLwBCsqEDyIHPaGjUVDSQpeMVoLzgdgKIlWmJjFDNTiEDmojXYlCjyoHSRlNgNSmtUaClRCIyOvOJcjSetqJUjiwdmiLTiUJCcYEvjHmCyUwmHskAgMgEqhjUyQOWuEsgALlpXblMnDcbuNyeOnVbhTJNWwALIiukkhlxljChAoAWLRklpYMzYtWsOwXYwWaBDAmumMzJeOfmZMsHiysuPZPiUbhZRVUvgxLPmNPHFuVbtExRazuagJyCqytnaCrSuAckxHsaKIfsXszpnhbkjLPnWjaivIXFgkcFCQLbZYYHWRnsIiZqDxXkltELsPGKeBhRiZgskfxiucoBwbRpTKhWugQEXVYaUJBqVmMKoVBaxbCchCZHHwQsBdXzcqAFchRAXqQseJnuTWXHacjLflUfHImETXmABOSLKGXoWtZsXEuSqnNSXRePSbrhBcsXesfxkkzzgUWMlAEzFdKOygSfJOFndlLsuOsFBAMmfvLDLxteYpWCtKywqbrMiYuyVGNByGlontMPvjxvnmVWZmfsPEfQpIuGHTmCwzQZxXyMpZLiPhLLKRVRrDoVNNKnfxjtOgzAQgiKHNNAPabvqSalrEoykQJjjrQupbaRncFSgxQsjmUFgDOtjGxJGJcXasJDOVWhQUpApYUrdeVMkfuDhdqMeSmlMBTBDeDVVDazeGZgonBYqPmUIRoPGlYmJeOifBnvBTtDHKyDhYHSXWhmORxxEgNrTpFWIASraHsIklHoXqQpNxScWVFfyyxPCexQVIMbWJXbbATiISEgETsiZwXbyVYmcLDGWCzBTxPtwWSzhZlAaiKonFqBjlVchqKvCjcApsMwniEbDvUFbaVVBDmreipcPnEqvaPOdiCwTgzunjjTRPFZfKhJqzwTjwlGRvPFWUMwoWTXosTHxvJHtcsCygTWaGyhKLxagdKyCJwiNgxEIxsREKsqARPNzlkyDtgsxGFZnHoqFgAsBgNsdbThIFtUZlIckuKGRPPDQDIiosXXcKozJUMYyiALqQpqWYBUgwycvYOQFDXTBEyYeUeDLCFogxiWpnJJIgvguUsViwdMbHYyvwhuCLbcIAmSPMtgYwdraSulrxgUtqFnvlLQiHjOdVNVvzmtpYeBbRstzmUASWcaRTAZiwITQwIsTWVbEUmIYLDGkYJbGChtxZgGnEkunpoJhCbwAXfrXZtIoLXbkbWvonjjuXLRdgLNngHhkWhEcjoQIsKvcLHPCclVUYbTqdmPVDoPNwVVTnoGjIqKnoRZpGfAMSRAFsxVStMbOcUhhXBxPuOWfnyGuCuclWmurJHIBmKHaWACqzmlkPqvAeJbomWTlAKgtlolVKRlmZtGwoYSzEtnPQdOrcSTaEwUTGGshBVzsROtmgBfZAYEfUSPGYuNtjTfOcnBNjEsPWQAhDiBKiojLvIOcSMzwYApfTEgmbsCCqegUssHdupxhZyaVBnZWTbRfEfdKfUmbEjrtTTbJMNJvTyRnUlQldzXErrdYFNgXdXSbHjjpCDuRbukYlmuWPdkFIfbKnzEywyjfTdYCkWtIoGsYIlVkGQoprBVYGnvkmBWDUGvBZeaGRCYyoPmJcIsxqQfcCxPEvpxjByIdiUGIyjmPxgsrrxYwuRyjZJJSoSsMaSFzohIzCKuBolrPdZWmZdVfQyMXNVAvYJJBJhkgQGpdCCYrswZiFMiJnpleWHczLkTPPZJJKrAuuvvUptMjIhYTafEiwlgDHrQTSvbKFQrIVAOrxbpVkzopjJIJWMyzMtoWANqIRDxeUNRPFUNJxbttucfOzzdWhBqIRIdAmUQIBGKdykBrlouAFgirATsTsJjyRhpRQEgJFDywEAQPmwsoGBDuAKUdOfzcGqvPTMkjesPLnpqeZCtWoUkrBizObDzfbVhQvohAMhdZPqtqFNGCmAAXohkqdntWZFZZzwDVCYOLJfmnhzmsdoMiIISXmNGVPQgnIdbvQguyuMEmtHIByyGHBHCunOHQXOsyJhBGLKiOkdgNEfOQoZtOXAaBcVroBDBrYPnJeBlZugGrOFFfzlMiUezZllMbvldesGZVenjRpLkHxXiUECzxZGkBCUKKtfrOFptNYPYxdvrYnCwDozVsDixZtXRRUtZnLrNvfBzWmrUMWyolbXZfHgjimcGCCDexqRgfLbiicpTGDXrtdJZxNuWONCcTCkurNmYrIseTUTfrUdAWuIAiEcKXVSzkaaHwjUKTjvgBzKLdRJgHJrvooagEKOMxdyXkIIXWGrIrzDiwzukanufCkIVuzIRFhUNkSCkSjVchyFuLSqairbScjIRjFLEtKqYbwCwspTBckEpOBVgehUGQQLwgkSecQMeRYACzKvYEChGoZaYZOtSvMBpqGhlFpQcPAgXSQkZyPEEKGrgXJqKSlmAkWzuwrVGXgdwehhdNYFhCjdHviMGXYeIqtudpjomfEOdBAZkDIGnmFRgkrGyCXQRSSoglTwyzfXPPIKchUAuGKFeplhLwwGWXYLiBmEEWHndfTkJfGjSfgRZloaMjmSYnDyJEjvRQfJwbZPNWbtqsGEZLqjQUHvnZxvlrdYEdfXZKqREFaCvARBPHfTKBKwXIvUamFAbwOPWaVbZciEyzfyDcLgEREYBytWclMHiyVJvsMOngVMRHgHtHMjcwjBoJcaAzHVeuVLMGrneuAuGjYAdchXETyGHZaymrLhbBFEbswlqHDzaPbsPTMeTpDzBblqvxRzrqtgYzDALLOBhCEbDiLFYXiAdfDXmGrbEndfyGARpkuMOqiNAhqUJaDMNJTZXnkDxJQGFFlVLaSUyiEPcfsRowluYxALOLDiHdckgGVRDYMzrEuHuCQrZCAKZEFjETMudiMkransICtNVpmJwJEHpDLWwykwjdtuxHaKmhgXZJPpDUidpeTVxZCYxTATUMnsNuboyUUmaFLtKkJQbPgqIFruiIcZgZAQZLRFIdhssQFvTMUToaatvvmxbppcnRCXjEVVscMollQmDHOpiSnhsEcvCcxghZUWscirJReakQnBEbanglhpJUwBIwThqQAKRSRjhjXXUoHKjdRQNlQiSUaxjqfKuDXGRIAlVArndhqraBbARGmrPWqnmDkNKfEegmXAFsHapkTBhNuyKAjJMpvFedrBAXwlKhUcyUOpKIHcwuqkRyfMaEkUtYHoKODojIiDJVODUjbbIiKSfBDlebgucJEfmDGlwFdUySIAOBvzbeYMEMveACPVjfWziVmgLMcuVXyUAxIiJMoQgmADfuqqvVojsSGniRpEqqvpqHzlJLUNGRDcMwoGmbIwtQOvKVMkFozRneGLRnFgAbDYjXjrQgPeIXJEguJPrGyknuDqmrwVBMZvfbZWLELtpNBkiqJVgFnRXRlFWpZgntZGkyBbWeTvmoZidWzrWegvYBPUQxLNPUxWHCGKiCruGfemHpKqdCYZwlbhUdCVSdVgUilLlzURcAAbWyRAPSxMkaLUghDbmHImSLDqQGyliwEraFAhzYHEltWHOubTHDgQjpaOaOpZobRWGopjBuHCnxMYkuzIfMukDiRGfsfnzPCXWnQPsLasFbHTstyFuKugaSqSgczYigEzKTVQPTcfBHGyIwiHBZbfFlmCHFDyzyqyIQSiTevbjnHtiKakcmthJdZLfuUVeFlKwSNayPoGfbURyPbJcudjbCBydULUQlNaunOnpzXwIDjRDKKQnxfEIYVhmldJChXqsfgvHaNLMoKeMVeALbWmzkayilHxUblyyCMuPDcSMFAJvPgWfhUcusmeWklzBxZarwNkAvtKTkfIXPBcxTaMeubvJRooRYLMNXqNFQQiIZCUJUTXtjOHcnKYxiGteisPzGPAzVpXofhkOkHocBNgXNOBMxUyOdMrTcBZoiljmxUwrfcFIwxNLGMzBlJcqbkJXzednLLVgHyapiqqhmcAHfWuaqxcsGJnKBOdnOdbYAKIAeddGkLzSRmrMgrRqGPnLBlPHSekugFluSPCANcpKZwXedbXXwlEyGOTcwnnmKihQYBUPawummwfkDghMWZvrHUTMZqPsbsaecsVoDbyQwoXoLhmPNuIAoRYFBeoQcQgDRDmMDJiDEOmhswnCBXJCmSlJxRgiZLmuiXKKHzGMMjfnifCulEXwiCEUJparQzYGyQuvlcehRPgQkqZOpSfntpJTHwanCVZAfMkhDbWzTuAvVCCClZYXDWFZdOhxNMaMkRRzGgVUebvKPtpTecWjwPtgWeBjgOIJMSFkpVQWebiVvKNgcQNDVrlzIMUzZGwLWLwRvnNpEYzVEWHZYkhaKJgjNhNPvcIPnrXhfMQKWvjhWuOOdWCJZObsScxMxMhCtgICICHrRTgMAxptRPNAHurJFIGUXvUHCRIRmIlPbvLEvlmBCGIzEAHqoKskTEpLBNcAmrLTteQctcYzcOAAjWijdRuKsoQSJUurtEJIOiYmVVhUwnBWHWSZSJowwbXFcRmmQHWadnciJPOCebPFDfZMUnUKTfOylzwrCLhRqWkYZHqvFKxKhkdJYQCakfgtKVSLLtjNwhhcoGXGlENxNLnPySdDMWfPrTSvoSRPxtsgFJNsSVCvjRgyzxPEJfKfCvJFhaXrGQSDaPnZuBRIeBXYRREjhNkaSpRrgwZVmCMxzTdvDDXbNWLyyFhIDarHnafLBFzfrJZMjMDviktFNyrkCDOynKjQIAoqzCgiEgyzvionbNzjtMGRCRUdLJtzTOkjwOfWdPeJzTkYjqUksXrACncNMrtfHTRuItDrJDsOfJyXhUjDpSIrwmocQZlMCEKlDxesRYvViilZVRjZHgCEicbIWOfKtAnGFzBbRyQbQIDkCaAOBoAOBnUvBtKIcMHyQaOnVpOuQxhVcXzgUrowpQuyaRuNQuJbwHTcVqxuSIcEwRFmhDNZKLslRQXjOvllUherUydiHQEWtxTiZlQXCTDsxkwbwFjKHYolauXzLddEZDXwbcvUUvohsWuNWqlhZvHjvnRusOqvlOWKhjjIGYCVvZzXSZnHoBiXlJMzXIOQBkcuEYTYLhoSScUssDDkKnwfhkLTotPPBLdfAHIPPnvdhLyBECWOwuFmZTVeGtxfvNtBLLRqmDUedbbhKJVlhxfhQPINExPlssmkyztPAqsFTTBXFsQvfZICAqcHMHRIxxyEfMqDjYRtkjfFcdzPGkHCacPWbmHRRTHhPvDjsyrdFvTDXZXbEupXRIysjdwsWnxiLfnfovOfSNxHJKFCBBgmgmEKzaZRZTcYbeYsAlRHYHQUpGNiKqFwCTrgCeJJDVOHGxSOSqnSDbAQslQXUCSIWPXbdeKChvtkxLTWzTAbFhWLnoPOuNuhZivEFeElejIUjuajvuTlQjXIitRSjdCqPEgrTeKVQlGPGajXXgpvISNdDZXgqMEZIsPHJTFVKjGMUfkLZgzCoHpAYUDoZqJSpUCpIUfNxTNIfmaBMgXvuxQkarYFYAvFOAFfLmGTibsEkOzQkfWYQBlvpzMPKfyrtAjyCeMUhSigquKBmFqzvUFMNVYXFeczMURnndzUmgfODmAjKrjCFoAdTZkKlJegwkTjcRDCsECCezotZESOWZgTCrFsPpuThRlWloJMpSgWjeKbmjJNWSIlLdSAtadIYSjXCUkRfDJbUXKKiqUrqNdWKHEzAdkDuEZdbDoqDdyTwyZaOhGSsnRkaRlGvhqxtQMHDrYFtNUVVIlXyCRmgigINSTcNiLEWKGfaqQpbyxLtbXEokusMcskBTVdsNNZBAaAqonSlvmJjHTGekHGPTPaaMAzTaZApvCWHttiabUmCpPPQNBpyqpbjAJjgSbRHYQkEyUEnFCaSpeKESxPmcNSBdeDRwttamiTzHToOwCbXofwsPpgImsLvJuoaryRxWfeqJelKonbZQVMbJBPZNIpCCbiKsOsCGgbOLlCwxGoxwfEMCAaGbnGCOqENATsZeExHZsAVzCWZiPLZuxtmSfNVWHBITIwwoTwHTmrxonmPohBTRSgJDflbYmhfjXfylTUJasFxwQtjBcJcXESKArPsCcWchMuGnFBqhniPJrSZqzheDjqDsqcfnvytRtbSZcluLVIPqNrLxTwvQLSdzVNNjybhKUSFraBzUeKdLgDHhHabOrNbPAHogNlafDRJNFPtTVEcHscNrfYBePuLGRFpxxxxsWQYcFguMpedrxDibxvqBtEOHURlLpfitERtZHGCMpsaNyketSDwOrbDYHkFKGmRndIqqJeKcJSBEeHyBvNBqKvMNHryoxAZbTXwaKqRLtCENZJaQFqfCyzeBiQbaIoaxZmErfUPdOgQPkIMOrKtmHcunSpZEsvJWFdUqsDpkpvloyLZzzoqLaczvxMxngKQBjEmPcbjneVEGxYskaWzWIZDygSuLAtYWfFnpusQrLOBhIEFClPBptQNKtNGcNBhliWgVgkyheVtKvPRXnLpbEvLrqpecRbBzCKgQQWcDTuMKOnQPYVbyHqpSlHUIeGedrUxIsjCeSgrGxkTIQpFUdQyYVFDeNtwIFciHdpZxCAzPfXWViVmPYNsjsVXfJuyTqaLBBtcnJqyEuWADiFrjROrCEDaaEQzpZshHhzmlrRyjwwacoCzRhbIthDgysmtjcDYSwedIdrqaXkKpfwAxRBPABICTdSNhZxheclAJfyLNUKHVXVHvrnxtOgPUPgzktLobrTzpWylGgEfiIRbwUmBfmZWBmvRFKrWonYrwinQqailzgquNSGUBAdgwMMxRrDvAXjASPeHZqhfBqZEJwBAoLsWlBWhCJFmEVehcYFIGlJNpBVesPversetNjkfBsGChGfIEPjOxvxXgglcEKVxoBtGcugiQnmNpyjVmEmKMtHrWIbJDGNCUQokUMPnlTxikHMOEcBdwzixnYgChdqbTMGcOiwmFwNwFulcMOrrYTztsMdfhkvpmSFxzqmRaVDRwBhgkbZkfTIOEmwjtQmBpIUXTiulijXZETeHCeNkFDCILUOtNkXFAmEiAYXVpkCDfqCyGAqOrPjuyRXIwRSJYUavyLWVBLOmxPBsddYLzGYJAOeJKyPjmgTyYMZuKupEPdIWvPKKsCMrnKCtvxtkpqIoiNzWLJUkhGnPWXwfTdNJmXUUqjlRLLTNMQsFzUAJxOZIvUUtfOEGzESLNDIUCPkbMQyQrNDlnfykaZOgokwoxzYjfBJSuuEmLLydTvPtooUuocfVnPOfiKZZuBnqYfeMjLxwLXCDStHddnWYjSFJAixfoALiWWFQAFPWYBENSyfYJUmuLdtauAYqiVqDkVjRbVntlCRePrKyqkMaiIgiUlZQyGbPTHNovahQbhEtxKVznxoFVdnHTLvafKNyMxxDAHhzBFNvGlynFYEYrLYCEsmItiXDQybSMOrAOIPAAhEKvdQVcrafoQGvCxNkoeJLnRQsIXCVowxzRAasLrgwlnEMHWQoDcViLIIEXIJXVvqvtlJlOzKEVSQfSLcvGxsOBZjcuatsXqBsNmJuDqyvIdevtfxyydvsPFhpRxUlZgHxPHXnEwfSvYNjIKqoikGERhQFsqpTJPauSTixsEfSLEoIPEDCMHCBxgCSTdtAxrOscZWDhGunnyMKFOjaFAOoHPzTMveXkZZzMuinrPEimxZZfJutyXBrKJSIfEQWffQOTgcJodQmhtEyGsTWNQIpDjLrFQYXnDrYOeKxwljYOfdpqOELFUSgMEylQoqEqznHsZdEBmEBmuXmcAbPpSkBpRGBrnBXhneeibemPPnpvLobXUKjraqVHxLLzBeCRUMjAIlXLqNuDQHVTQVmFYDZdmYmwySzTagSUTVuSOfmUOshYUurPzlMjNDfKKgturoYkGukEzMuLCFLaeeXEpFQHAHAiMiBkGvdExzSXIJXwcMlkxeXoBwAFCizWkYEBgRlFgNSYCVzALhCiBTcsvbtPuMktoSErZvlplWCMMpQpIAGZqSVRqwdBjjzKDMEmSFEAOICFoOaRuhCnxCvxvcueacsuLWucLjTSOqjvJGdKJllRwHQQtvijcorTugclClmGdmdxEPTdSoGpozjMLlsYfUSoDGBHtVErMMHAXHaBrOiYgTmPiKLHTulfdnGuvxrzccAHfqujuPtbAluzdcMpghLRsAHnQEohYWvMZfuHItkqtUtXoAPdHKvlXjtamsOOQsPLSmbPAdRkrtYItQnTEuZUwJBUAGjgWJogYyKkjfHVdbbQmUcrZAULLdEwNvyXpvjFBegwkHMGIVUqkcpEjblKsbPdEGIenIuPxnENhNzkPLozRNvynEaSubgUXKJoYNoviDdnnQHIOFmKAMvEmRMOIFUNfoXaqRvYqrZppaWELteRcxikTjFytqgUZjRHqYxvjvcIYsmClALBcsyItFoKOnHhBqbfMaZzcwFNicYWjVjlvTJCwBBnVfmWpvYVZFIueKBjxAMypQZhxcIWddbOkayvnCuRFulYvqlNSEkPLkPVybyZGjsEqThzClhEJxNXuDNysAHaxGyjNpmJbyzxslgcXGCZmuflVOLBTkOpuHQPEzsmkMmRckIhBuxsmZFybZvMMRljZwseTExyHZaxOMLRHZXSmCXuEKHkCvBGUcGotGgWrBuRXUTDLgJnjxWjJlKKOukpeOLkxkXiqylkqxnssQdKLchUWneEXMgggzryATXHiMqkDUmIYnzJclpyRdmoVKTWrFXzYOoQwZEOCqQOLcANmssyxbdSqowiaEyDwLjKEZtgtdAXkNelMggALfhpzcCacEhTDdQjSiortapJayGqQDhsNJJjQFynmxchBRQWlUaubEWWTVQOaPMFHIEYHWYRGHAEZcCMtKkgQrBlsaKYytPhLtGGLKRvbjcYmGdPpBgpZQOASRQaRkgntLWloxdqeRycUDSzZQMXTQXnRtqvLYhWacycYDXhwwWmnoBvaSlAdaXMLSnajiqomGJqMZWiCUDXOxdHABLZwTWKaEbKXZpkEAGVzCXkNKfNEIpewrXcNndxQgwjxScVetynQUeDTJZkkJYPGkMmchEDOqSbnsscEIMUQeeytRTNGOzKWPnalOpeBhxYaQUXUfsinaoEFSZTlQdqFWFywgcftpPNRkRvYJJbykjOfuYwdOyoMlYGjbfhWSDuEgfRydRSlLWFeHIKftITBKUipoDPRcqPDlCfhyiufoZjrIeMgiuIsibsjPLYjNuletBFGfHlROCLhgmVDaBZVfzJhfhwySVCISzYLLxxcARjeYDlgSDABQzHKXfExwLscPmnUqThGdHtUSlTOKioDslKOwvrNgjXPjKauViaMyHLBkeGWEOrPIrKWRaGsiZmbWDzPIrLtrORiOtoiXteCJboihtQZaoPlhmOjApYDXZEkqyYVZPKXiGwbziOQRHqRnstdlbTYUPNCUIEGRHrmxCUoNQJCYnYlhUkPvxkDDxAjVEVDdAiKDsgybXRaCTvHCJAePcSWejyxSCFwZMOEZNsdIcZtbOpRYcSMDktbPeemtUpZyfhChdJbQdAwIINQvscDQFZnideKwGfxKFXWwfuVsGYdgzHlRHobuSvtlAAPvNYhwAuMEbbIGEhrREKHQNNTtPIAYtDJnSbLZzGWGCnzrqXBLhlnIHQXOCWMiTVMwjjSOCdXROoNDrfAzlVcXZiyXkeCCYhNYwsItxcigYfDSkBkqIWPBIvYvEOJWqYtNmGGOGelgXQsmgwWYdPMJnyqhYMEgHPTvLIQAhmgWxyDGEVffYvIdeBNzydwOuSYplIFqiqpRCZFQhONpHwEcgPVMUwoJLCctiKDbqQTfcTCjfwhYcftsjOubkjpzvsLpXihQHguiUhIyfbszxvpALTzFkBOuPtuDfwVYrpAiFLMGZBmKfWxqgosJohBfEmSSCwlVoIaimhTwUPaXVkYsPgRCmGiciNHvfVpHGcuWfjglqPZUKaQiOQLoLphOYKRWnjjmTtvNrsxPghwKyPwXhrQfkkIrLbnClFREjKiUrjMfiIRcKkmQVZRIeBMiTxWeanINqSBgXwyVBBGkaWkWHMpfCKNDUagcaIPrIXmpyEqsHcEKDxdKdkwqmXDVengwotexSoKuQhOjkOnOBJRAISsjUhwvaZDLLOlZUKAwQfKYJutpehrHjKnrJhujqDTRNQCVwiKYvgQriYBxsUALuVkZnOyWpOQHsPuqarjAulDwNohjQODSHSHirWCCmbYkMXdsIoQTqNbkcZYoTSZmlfSBimdYuKhLUSxlQreGrxGAdrdeliKddwIUEfSMCvYdeLGIuePNBImesdXlHBSKVnuOXYsMPgJiTvxesZiGkWrGPHalnsrxxyKafiTfDcOdvVjKXYQcaFaqMIkLTjYkqJNbWfXFRPiRRWOHpEWmaJiHfzGCcWopToTAsIjLjuEcWMCZnRuyqLcYzzkTYykBbaOBGytXQFmJRvAQEPATwpIzXiaAElUCsntXqieYCDBIMwkWFgRyWZonrIWsftbMxVwtdpeTgaFdFyMPcJWwkvktOSDARbUGlzuHmohXtbeiYwCeIvYnntqBCgHGuvQTilwvNGztTRWjiIwcrnjPUFDkfjvGHcMZMTmurEPRVOjmgmtKjmyYcyVQeSoTMfLagxlIMOoizGOBLpkqdSmSaiKJgixVgtHKamVBfjujIYIgEARNedYSXIobuzUDJJngZvCgjMYssDxPGtBjyOJAmahaTJbPxzYNnqAbmInoifhryzaTCBBPKLykxzJHoKSJTMEqFuBxvAJowTMALGctSfpUAkoAMMSDgxhssxWAQRmXjapXNuoxEeowNgjYcVxUqvvpKeVFgqfFnPkaqYePTxwlmnrMDSIPFRHhBXXWUFIGtcaoCWrmfGMmLUuNiPtNMpieRiuphpAKKqqZitRUwCYKPYKjvgDUoIiPNrmqRPYMwCpaEMzgLSWeJdrzZxYNEUPLdTXNsRHtUguRAGbkvgGdGBevZzmSNVenfZqqoFkmENFKHQTgURNUKBTaFKoeNUHgvaauwdkeZcYsMFVxOyDVNdwteGbXUadRjcoBZiGFbEQLWdwFivQFSspPjAEvPQeQxcnOMMtVUzEvQgSAiDUwiTIxoKGcAeHcMaoqmXAoxptNHRffBBGbvUnNlsQHlcOXGPndZFkuNvfERSpZPYDJxfSUYLmuJUEfzXALBOnMXDahsvURFcKvuwORRoMEWzJRMUoXhOvfuvURWRqfknPonKIygTuCONxnFOveZUOCbLjmVuGmffbIlMGfwPckBBUQLVDfGFSuecTwdDhPbBrGclJihFhqwZGBpTAlSpEgdWKqGvygcHjxoRQdmBrGOwWRjhFCIWajwGnrdhakHtVjNwPDXZTHQdXVYOvenCSDXkIaUXGzPVySXfNsnwkwUNzVcHglizBqxrrmTfZtdFDOXEgdAqDfFevVzxzQFoEfkIhjeWybnIKDFTPrsqqItETkKcVgyRBTrytAGbBXvfWlStcLmjGiGeMiHYeydMtlPFeoVLScmEntIBpvYiZAtwzbAWvqIOuWLEBbNzsLiMfUtKzwjcEthcznVRWKBRruoQfawwkFaIBwLFhhoQNcqXNCIkLjKAljSIZndnvYiPalevNWSfPDEndNOTVRjPqvaoFJWIAIHdmktXvfdCyXZTjclqreqgpqMXuSUaEFvVMyhHBWVEMQtIvZqpnCjmlCaYqNaaOgokcPhXVWJrbiYmBgGHFGHPdzvlOEAJCJFUcVidFwEUevrZRoeHZYzLHEcarfZDyIEosnXnPZuphPFxOpmmUHFECezbFvtqmdQWBBfAIVcqKOoKMTejHYEFVOHMXCHfetyhAKkXfjrstNseWJrlBYOaVFsnqfbiEqceCCcpFLeCWjdesztcqmmVQlivbwpJfEcIrqyxHWKztWxWjcYAnTUeKXKtFJfYDzriZlRRWJvCTelksumDrLcNEFsQewOQYaZlvbYlecPvGAIzgkuYYUwnPdXsnGYVjYIyOSVhAwPSBAYmoLjbjhMCWUFvieZELMolVKGAlfHlAOILAGpAFlfmzqQOwiqYekxWVzLMFVuyPcvjEKwBPTcbtZbcERNtyQBLedLVhpoWokiXpzbbixbaWeaUIwelfdkXgxUaUOEmwZeguDlNztyKIYbKzdjTxbeyYZgvDOufCyUIfpKOtELldGKfJuaSZihupCWLAPPiORVzxCqiIkgAdHwSfuSIMeHRkwWxDbZFeIQxENdlPsEHKLKnkzXonyyxYNiUGCdFgTZzdTwGfEBqGDFtYFfXxFMPIQZNqhaBszkRxnCZXEBtkyAXjkewHKfEvAiBCisGDOhKfNxoybhkaSETsERPfQUEInaJtHOqGlKgGhARqZmLJbRGajEJZIximBWkQyoaeZyTMWWKYeFQFzwXRabbKEjZuCcbwyWracSgUEwmcHxPMPinxZnghbwqBjOlKaonVTcpVVareBByMkqNOOHnvdDcwYmlJRTpjoZFVRjNlXeOnFjlbHYfwzLnVyppFUetESUvOgdQxuTBriwUAUVmiiTZXWxksChPTaTfJeiEdzGiqTUpuUxtAMTCqKlcvXmLknktjiOUcFuNUsUTDIpkRtyHNZJSoEvbmRSCrQKZChqlJzmRzsbRUPwqffJhdpYofwYLgFXaACMXOoFzbeauCdDqtRkqUWeqqcQTBXpegQpgUWIccIWFQCacOFeDsKIVfzqqrkLqIvEGKmenSjodYIYSgihPikpxFJJZbVTmHxWTteezQweYsTmqOpjsJjLksPYThuanygwrAdBgDJeEfVeOJDUarGSshSKtwfFrUVHgEaVJnlwNAzTeWhmFaFcHnBxibLQEEjBTPEchkUrMDrvQwQvmiarsjYJVFJafCAIUHYEUJMzkuCweqPkeHSZEFsmvSktdRcOjQPadMWgPFslHaAThyZoxWalVCHPTuTmQVfMBPGlWZnSAKBnDFxWSLgsLzEgvcbDDULgnoIPXXMdsgHuLotERXoPnpKNKeMnfKUpBgeVJDzRbdeAVmtGGDwdMXWMKYbbCpsaTTZoRpxlJcqEvbuyTfThoWBTpMJbGmWnIDTFVCuHRFySmBBjXOsfWLyaIRmKlJPNpLznNPnUcMnzfEifSnVeqJOzixtoqkENAQpJyikJWFmsONtOsIZfzfuELrainVKWdfHgokcoaPBoDTFGwiEiaSNlWJoPlHKxbtFfqaiQiuefpRBAIrVWkOJNJHWmWoCruuUChNSTTkgNUsxnZWOclYJjyxqGisvgZmLaFTiofQfdTvuEylAHgsZJOgbcPKYySeYewnnhKYrybYYYvrljFMtsSnGQzYkKBlCjYNJaugFtQittHPuMxKyTiZftcJEgBlLvXoxhiUzchJflvptxBHAooMlrwJnOCasmfuqHyzclAWVatwDpVyOUecBassazDiHBKxAxFCBHPhUFgVzsueQbIpGdeHJQhRjjmxcmlVqAgWRBhnkjupPUKjJWWPLzbsJstdYKErtPGsRTvPCqJlpxlTLDsaOtxdZWlggsZOxglXZMntnSxqmnNBnyzvQkefdPQsLBnVRmMyAgFwIVxqdlPaaouoFaYeIzKFzkVIqimuEdbyWZxxZZgAZFHfjShxierFCRePRWWiNkEzsjjcWVZLIvxmJZzBBPVqJlDKdJuDawdqzhFsCZeBjZdmpDCXhjlpwoClXrDBmwXypEOcpwtirkxTLHdyXcGqKCeutkdLYoUYKysBrxUsuHIDvpzfowbbiOuoaiTuPXvbTVkfhaZieMwAiFTjfYMWIMkxRHsvhWixhMRbOAdJknAeIVFSFyFdXsfXZUBBTOuMJZKGzWhWaXikbDvwhtvpcZJFCGcphHGOKJEnbgJRWninFuSpyTTHkMBvttoqtrMnsrSiKUPaPPIoJXhJdeYcIZzhwqWOzOnMDuntpwxmMWlryTOpUGqxRkxDIkddRppnxjIqbxOAoOamWKywUimTbvCddzzDYuWBkLnTrIjgdBDOqaZQQedxbWOIySrkdOastuKXmINHgVOfhXKQyXmWUlsXGqsxWGJcjZPtKVzxYfWWNywIshwxikmgmnywUYXZzesmNWEufdcxsqqkbiaIDDVvnIpUmtjTUevdebeZSaXTuJiDYfUDdNfvrGUebMPCKAdhNrNaDUMxMlWvTWornRyCLRHIBxhGFwVTAvKuQmRFHYpEMafiOvqTgRgaSXOpIVLMfAqWWIotLREEsnpDOjwrkLQtcxzsAFYZsAJhjUcGIGVnwecLubdNJSnnIONOnPEqoSfvrDRuvnyzQLjEpLjCuckCGJIPeCbxiOVyTXbQBCPBBKulQobOasLmyAZJyHAAcJBeBFaifuoufwcIrAQFgbHZSSIgxVZRhzyOybMsvOnplblokZQMlDFWYxpIDqWGzmtDqHxpvnKPgdzFCZOhIUvMHaWSsTCmkiVRfsCnZOIdeGdYzbuwgyTaFZfbXwwEstEuLVLeNzPjfXKOmbnESqRFXJmuuwhRjlOPPSVSnJmRhvvuDIHFTGfiaaxyYFHyeKEDbAwqvIWAymTjytEOrBEVljLSqqSkAoPDuxWVrTJiRdqNEcWBDlwfAZiMRECFvHVcqWMGlZbjOKRFTCJedsBoUOLxRpTEPQqJUtjZJCuEeFsDuARZeerVRfdomvmfNGNkwjvtioLBZx</t>
   </si>
   <si>
     <t>2026-09-05</t>
   </si>
   <si>
-    <t>23:25:35</t>
-  </si>
-  <si>
-    <t>2026-09-05 23:25:37</t>
+    <t>23:42:28</t>
+  </si>
+  <si>
+    <t>2026-09-05 23:42:30</t>
   </si>
   <si>
     <t>{"key":"value2"}</t>
@@ -371,82 +365,76 @@
     <t>&lt;root&gt;&lt;key&gt;value2&lt;/key&gt;&lt;/root&gt;</t>
   </si>
   <si>
-    <t>9223372036854775805</t>
-  </si>
-  <si>
-    <t>YE</t>
-  </si>
-  <si>
-    <t>nt</t>
-  </si>
-  <si>
-    <t>XU</t>
-  </si>
-  <si>
-    <t>hcHyHSvxNCKwadQCydFjrXhFmiTPrJSuHkDQRGDsHlMvHUAJfXQCcVbkJswGpvuIDQvoKqhoCzJZBeTFFTcCjWmLBwdcWllmRAYOHysIdNZUWnRkGIsaUqvHeqmGDGVGqlOBwiRtEwLBFmljKwuriyaZUiWoHqMmtYgVIYBDZOztjNMPWnfmwDMUPrvDYxNHOsCZOIPLMXvRDusNWjFXRAWlX</t>
-  </si>
-  <si>
-    <t>dkbSFRtKFfSoUthmyqSJoeBFAdFOksBrJxJgjzIzqtnwPQDyNCviQczUaywZZGoOhQtoFobbdtAqmpHiVudRLrVqXGzIdEtMiNGfzbBShVOWqMpcbOWFWWCTYKjBBSSZNwQKVicnKlxDpIHRfmZwtjZJgh</t>
-  </si>
-  <si>
-    <t>jCGIdNazJRVowDqBOVlKXGHiWoVaMRBKkRSnPdrevdAhykyKDbrpzsybCzCPjHzOEIWOmnQGZTMVdkRCuGGuvdeNXsIWijZsPCBLSPPluCpcnbVclzm</t>
-  </si>
-  <si>
-    <t>aTbRQubvHKymvYgWehHGabAGXKXLqKlKvYkxGnsNopBZTaQAMFsdOuKQFLdUXfJXlsFMggZyKkIIssksvyZpYYESoOzUGomNVkQuWjycxZQKRsPMoaXwBwwrwHjuMzwSuPwGDeZBUQUMrfegCLtdzLRyLmTILPUrwOOGLyvvTtusROPQjjNZNZkIvAuoQzODhDbNJbmYBXCaEgkvKcCkmItwFQrjjbuORgOcFNJszDsSiRgdhkAmfJcyRUwLnkTHtwgtlkyYrQhALoRaygGkrrUhbAXVZoDMDzCAnOIwPWKppEoWvnQthbecinpfhRDHoDoOKxiivpjWkNTrxGNLDunTyVtnoUabJwkkVrBOptQYlrZgJFXkQwpgtOtGcyBtGvIqBPTNeFiQPqQKorltgRqyyojzDVmCuRbRbYrZUSCWKazOlFgJxYKClKUxHnhKBhgofcphJnqFxhzPXhgNoPnOtQGAllKfWByXWVQMzjHvtaNfXovCSVPfcyyLgsHettdZVtTrFmRAcgOKjUVaGWauwPAlqtulGPEPxVqkKBYKABGvkVIqTOTncSETyIeGMAelzQPKUoUzutrwRujIxnJfSIFonVHBnusCnhTjHbLFYmslvFwZYnDOFCNQpJoIwQMVsrnJqHUjbovILAEuUQhLksCbciZiVKezQSBCbWJLDHFgGOmOPrqHVBlltmtvbIJwIVeApzzgpRPAqJBQrqNXJmiHHiDnhjWlJgDkOkNLpvvzVZxCbgxYReUJRSLdnWXWuiTrqkjrzAwHLJgMEeavsOuAZZkNpEHepGukexEHKZBqUSgBQksYuItPxRfvSPKYRjEBDBhRzKyCpSloZkUezvSQnClLKYQNsnqUlUfutNqJbKHlHQwAPglmUMBfBTebxzGGiVFBCYRXIkifIHwdhQDoYcgVSQGgGrTYwkylAMmCCKJIPGFsBzZckEnGMBKyeLdaWNrvDjhpwhUCWOqOPsvPZfQaivTvjvrSIBrPemaditaojomowdwHfFmESlXxddFWykKdqQDYwHXnsEFmbjHgtAcngeLCwQsxYaiQnjURjCUKZRHwtJDpVlSchoFNWvRfKqTpDAmbbyfbuaydtwVqxlDBeLZwSMcfNifqJatzrewGOYFoUcvsDdBhqdHhaomYnSzMEhjesWiLmDTgdpciwqsemDvlAJGkMVDopCnuAcpsRqOISAQQRQJqVbRYcwPiNXHZOTlhtICJDCUsRalffhSganGlBQDoACeeFdgpAsDFLyiABbaYytTmYqnbnQfFaOjLGBkzjKmQVoleOfOjzCwLyfHUUWqLtbprlbASqnPPTTBMuzDGRhVxuTmvEiBPUeCVKHWiQUnOSvBqtXUWdZZWBOOLyLHlduWJsTLKWeNGeQZVyMHUWfwFTtwJOciTwxvBMVEomlBHAxrovWGlgHSOcnBqzTPZtqTjCJFrMgtJiPKTQWGZfSEFgHAEGOyBOmETLNlVPjCQBIAvnwhzkfLCzNhMikYWMaAuDUxMMeRwSAGDrGEECJgZmblHNtTEletwfhsHnHiAxEGThrbLlNebupSHRIgYZISSgTDNJzouqFydkaLgHffNtdHqxKAOCRBLJTKgHvghBDWBvGufkbcvxtuSPNAUETwuvyCXLrFXGeiIndUpcPlGHQRKrxofdjHHbmORTEPQyMEQFiKYKmJnBUNKkSggACVakBjhqgAgJGyDjHjSprjZxGWnPsNrFawfzuYInEuOvjsCuikRvZfPRvpVeqMIkmNsAcwxWMPmBQMPaUCywmPLQTsKkCqCRuOgKcImcnELczSrcuArKNjzdNfQTPsqSUUaQKkLlwgofyacPXWGYwOgpOIVjevapPyDbkUDLHxDGplLdRHLLTHIpmNvpLyyEPNhVhbWHiwiWmqjBYmLzPJdOXDcdowiPGpXCnADgsCvPVRlaZpGbHTsghvEBJDZsGZlTXZNONQRRTftXbsphVupADctRCattuOgWUovmVWlOxOyIjLfBilnMioTSgOSoAcBONOBYHJtGjgtmBaBqYXchRvlGVJQTDMoPMFOktpydQRTnvgSkMomVqsPCndlINcWUDVQRwtlXysrMZoSNtqbdFrcmvxuZNDxNmLNalSCiYeqAbXvPEDtbzZJIjLINsAawEZTTiiWukZmhnktaSfdlhRWwLSmDyYKWjXFVPDCfeMtIdDvUTgUMTiLkgozswWpILpNIrxGZSSxuVHAUMCGpSYWLXwpCQOqDWKNgytykBVIPcXlfgFSmjRUHAsQViEwQrwEmJZugdcZxkZGHPQLHFiUJwzKeekSvstxsuTaPGwqSlgQhLkjIkqhKYkFTMRKDPMzBxdEOycUGSIStNOokPamYgbQOjRrozrohqvCZNDlPdiZAIlWWEhvmYNqwqRaiaGPyoTGFMpNkLeIAJUPFMhwtuodfovJRUMyjqhnICvXVEgTUpByoGLgSnxeJAXruTOKPfKvKowLEjJuiISdOqQuiYOCPfRsRdKVmcpgfeuiyKlfLgRZjIdUmTeHhTrbmEfeQIrbsEaqMynYgmHdrfJQsXpuDPonpFwhHgZFgLdXWWyQLmuDMWPueSpWmSgZFpZMIKbZrjMBCepwpivfBtarxDhPkKkGvLlVsxQPoLeYXAgzHjmZVkeAuopxKuEXrbfVMolWizSOtYmbEmbwrpwJxlULAeObpasAAxIJbvSurWKnnofaNlylivpiLohFsmDnxGwwznqJDgZNpNIWFcpsIGaTNVCijFCYfOcIoJfSBLmbtvVhRxhFadclIAoOQpQfKDndkVLgzLdflqOvDoXOnxJBeCgqgKTEYApDBrGaMIHanfgxbhtGNsDRJeRzFWIOxfWnkJIAKnBgmCBMMKBTBlZhyHNhYYHqGuYPBVxLVosLYBIwKxEfewtwPeFPmqoyxXmNMxUhEPftBiqJiEyAeYIcHDMyXcLmEReFXzRYJguRFZkaxPIRbuEfZJctDPzJDjcSPBuHnlMsBcZmYJdRVqKHlKqbIwlrmsrlaHaMiNEabwllpcZFJXBcRxyKcScanHjZgqjryHjwOKMhBUvCAkaMrUyySjQIQVdyFklkfnLbbKzxWKPRszycljrCcKCgVlyrkkTHWdrBvmrHsItuUiCpTUyooCIwhCqgDPysLMBShcDWkTOSRPLSvNpFLbUvtWmmQxBYdQQyRAfzksQgEsLAmPaELcwZcvIZLSPUhWYKYsaHljHUlZRWIHgoWEuybXjYAxDYFKMYrtHCAkqVeOvppyljTdzKziMhALLDyHvbaVvLzQYSofQoczKOonHWlWeQXRYfBhgxNntUxHFJvqQIujQQqlPlznrwKMnUIlVCMXyrLMwrpxRCedubqcJhmSeXOMwpuqwGTCJZmBZJbtRzTfjRHCPpHVbNmTerVYTYSzdkXMkRMJsNCmzLRXxvWVcDErhKmlljeXiBWPpuowDDgmnqjqcKglRTBcsWCignLuEQtuyNLpesOrSJLpKOShqIAOPnAYGzLYCaIrnFKfcMNxaaQAoihimsvWkygAzrPIHNmdtBlnPhujFpNbOTfCbNqzcznATdiHUdsuteywSExkboCLrgXamYNtECljrfMhucAKExoPzwifiJkFQDMyIQbgIeFjXvNrwZojtATjhycZgZznkTAVlEQgGZVkDfsneFralHYxaotgBALDkiHnwctYGdRYAHSOqdKnOUGcBlEEXKzReQWxwyLBNIUjoHeLpbqaYFMSGsbQnSGQpoihcMtBngpahfdJkzkjcdSwrkVRjjEUQylfbNgkoxNzcrVQrjNHfxIebBuyUEHbWbtRzdaSEDHWjErrDnQYLkRChgjzsKAXKEqaMVSmAsLTMmMECjPSDGejiOLWnygZWlodVgjBomIqHRJGExupLulmpnGKETnOvqPSUjwOhTzOTMpQqOWxFkszKBWjrGsNpTAIxGdCqlkVeWgDnrkPCzeGNJNquOWklQrIjJICmsUnJKljKXyyjBVuYrowYyYocpyUPrhRQSBbXlPiuVMuJeuJaaoOJXNrZzMoFUcJtGrvqpseTItnrDrlJfAifxrUivGGNlmhblhkCDRjTebIRavTlQFfRMKgNxEfmFXyiqhMdisEXiGVzfylRLDrEAZmWSBorfWhMQvkHCrUCoXXBwrPWqwpdMlXVelfSjveNACvdsIApRjalqNGQatoaUgKgjGpAxZbsYHhJPWNsKDnGtKDcOHhtbUfQZCFeSSvTFxRUCSQVgQiuWdrfuIkZkTvRSkMXEzsioLqzyiBsglMwYLERVfzfcRGuPfwwYTomrADoJQWeSKJzQEDjXpWUkTmXTWwomEMLLJSDnONgqtxXXNaiDsWAUMcwIUuwBFPPDXHirSKPzCYGooDsvKQSKzxQeInMJDdLvLTJigByUColAIKBrwHvEDrEXDKFXHGpHQXAPXSTnBEwUNbhkOqLqVYaarmnJylEIdVpROXhezgJpmmaYpTGIAyGaBRuuJZjIkfNNfOwnSouvwYuSPxEJbCLchUthrsEbIwfxiMuoDfjNfeNBIGeujFawxCgfBsgneMqanlVWfzKHuIiyLZulyWotbCqYZHZawgUygJWzUCXooIOyWQzSpumgVrYhfWKtULWRrYkpZmHMbpLKVmCdhfUDTojFOqWPfKKoXhfXqQeYmoJerztcaPUBIoUYPeMvJxHvUQkkeuCrQPoFTZMetVnTLWYMOMJGgKNhsJCiRMULeDatgQcGAuWEgYuqNOAffJXmVFipxAZAjGwjyGjcJLukcquXEviDJZVmqAFsmzsvunvkGLDhuJzUnCReAGLFoCdRFUNEqKTgrjRsnBlLdxtFsmLBUHfbpXImLCCRZvPtPPMIswJBArpXyOLGfSDQrRQoojNfFLITQWaACuVcPQBavKAIGOSRrBHkfyNuoTobbPSLyOTSAmDlftJvzUVLAixgCeBRNcJkjwKKYHBDGqAlYGxmwiQFvrLPfUOwSiEVudXJRMpTKCldVzeKVAjytdHOvdQFHtjCApOrVKrWsCsadvzUlEaDtgXQKmMgavVwokfPDJberrflkhIccfgRLDgxiiYITahlfUjEBRqhxZCsHcGgVwOajQkxGROSkfIcofywdjDuMfaDczNbAEfDhuZsipOklVZQlvofHhwHvGJHeXwFIKVJQpVYwuAmMApGDRcPlrcbNzaqSIQkqltECyHLyULFdMGmSjaIHYpHDMkxfQHdIwzMKCPrvQziFitiMNHNUUhJNQhvcpuBHAfcKpnigFAzEVewVLakYzbtdvZnRhjdgUYahMvLYOFWEfijkJkteGKGULFapDNipoCmQaIIuJxOYTnJMyDfHVNRuMlqlQnNlUeLEklxsSQElrnWzpUyeLxeasoCuFZTugbWDVbYenVMuJIPSrjpviMpfBvoGQqAynxWoyXsJBtDcdjbIGtFAcQHtRiNHHsNlaxgFcqMwbNNgVuefQgikednElPilorXdSVUKbpvsSFVrVTcnnghYuCjcdZmXoufJCEatpVLhXHOcHpdqABZptFBeaaPbdesalBNzSEztQovwsQdOjuCCtxTtvXBsklEQodHBKDncJgNqdYewqylVPcfuumgjGNysVspdcOcRdPEQrAvxmzESlRJzFwBrLVWbLfSubLBCDTSoSYGxCrleIEoqJmnhnrQrzLtjeKcRusNEzIKKgyZyDGkmvhDBwmXtZKWGlJbKeQCAqpjFhEKcGDVwokWPEXZhAJyIFtYRvndfgUJpBsaSVToBCrFjfqeqywFBCCfhyGpybsiQXsoVlliBAbMoFaXRwNlGeAuXblZcgTXnGlXEYCmUBDfEOIoriidbNoHLjLbwJPwHKjJbpryfMsXwQfLqRcXxlthieTkOtgljqnzNTnNeDoHCFgvMAKMJaQxMVQkGIyoqHNHgteojOIBSgztRYHIbHcUaSfwmUenwwkGAZoyOwraGxShlWMaRLPJTiQIbOZTqAqODEJHqforVGArcGEORZbFqrIAcYYMkGCgsSdxFhHDTLVJoedFRKzPqGxzFYpRcoDkEmDaPnnPPyhJbkUnzVjxSFVqizBIAGgQxEvdCXFDeuelNhNtLmfypVpBtZXwpsPbibFdXppziARHqHvuLgLDnmCioeiErWbhSyuJENSYwofsgqVZAfpkhtuIodEpcWqylNBmEJAUtNrbmfHcUIZEvndruWnWEcrxKdBUNiaPQNDYBoGQtXUFUzuqQdplBugIrfJzOKgXUWCJfFJqYnAQOVnvXRnsYSsnsvkIeQtBAUnCWzVZzCILigtkkXxNCdojZkZGvjVhcmgjbnyyRnJzsiXEeDvZdzsLMRHMbRYjDJNJhnuGPsAvMKBcGHOiodzvyIDVWvoNutkCkMGeRzpoVssVoaKPwcYzmXQyEYomrdMkAqUpSnDiQqYNZjEAQZenqybPiyGOMOpOMifFTGmHROlHaafqenNeNODUMMkZuJJjCLLclFEiPQDcWfKkZWDgjkkkuXbJlvZGTgEMxCMzDDCQjdpOdBKTlJDvijFqgwQdUzbKKVpcokjrsZqrGoGrwZwlQSuCowDniQeJWlmyzJsOUlfxIytwEUuIDEvdWRuIuxAUWEukvhnxTHMLOEemeEkUUcAhPoxDXsifWkDsJdplPNULrfmrtRFBMltXmMBgqEmuIXFVTChDBUXTsxqOUttCXwlLUfgnVjzWygaSMDGbTRSwbcRAFLRarposPjJqNCYzoCmcpQEmkknuQKFlojFvupGgddAcRtjaLtqDnSZxgEuTaGNyiUDYomxqcZjblVJZxVwqDgJvpgnmHOlIiUMFKuNpazLKOWCHwDEQGoIiFoZGVMTTLDFHjsYgDAsTGtVkDDmeBbsKXNsQYYzacUaGsSEnXFHhxmKdBGoAssaPNreIwaFCciMDMxygpSpdrVMzEdclDMGzkjtOCCZzXjUPLDLlyRgzfLjnRaeJyCdcpkZIgcALgvRQdOZrdrzjwMRfuQQIGdCAeumYtOXHNYWLqgkkOiNWleKMjNPnFKlnVpNGbtViemeeNNGLfqDiYfJxuHDUvBthCBOyMJRYoAvtTatuQIuDKcPOWdnsifpJTzTkTOCiliRXZxflPWucKZobtabjRWoKOOksWBIRJVKTWMVXFPMRfgQBeybwmlShKKfBLEXcwllYzWHfqfmGOOcyyxNfVolvABbDTmpJrfcJNUvylybjmeVIaMGlPnjgkHzjJzWDSIZQapbMJRZvkJlBXufRhYeNCstYPdWEOrkqNaZIDIrYtsgNgbZHwXAbYxpqfiVFrvyLsMgFuUdQxWzwmfaSRLqGaigSxOXBeVpRgaexgSWTkjjhNlYhLjMoTlqEUojKVfTSLltKMjfaROXxxphoVcKjsiluLWeVCbRqplKXoMGkwxKOmYefVcWLEUXCJHwqdAVUSfzgjefEjVKkZOWitVDfzImVLHeQGIAetiPYsBFvAsUqBaDTazQcRUVcHAsngqlrwhOMRdZsoyhSabvLyvCVpknMzebATUMvqoIcZtovGkhDejnEdvstnCxnhSvgCfTpLxpOvlVzunyPKfjsANQZFmVRlfAWEyvJKNnvEVhSzRvIGGKIrWEkbNxFpQSgKzhBcCoiNOVsLgmwCTOVzrnQSmXKdxEqEisyxDCRpZTWdoZSLCqcqquvCyRQTEbifhyZIxfTSgbAblMnLBHTZdqaMSWGExcXeWlkceiQWYFJCKRLcCqVxNCAGTkDxSKmKXuiSumINuOuXqeYEoDOkQTZPYxVnpSHmxnXpINhDlzfhmSTTPuJuJDFfCOdzXNXAFMLCGMkNVDXYTfnDDDAitcwSbqvZvRicGubjorVVIZoHnnXEYajWmPRHDGbWykknwVicNOxOeqYiNXFbLrSwXjyegIsfedVpXRxGIwmGWYmbhpGbUfbMteetmPyPGkxbHgTBUojAoDWnUtXtgqtJFHrxzmkidjNaHoQEjnDBEasLcsVbiSEUMkRSnSVZuEPPelVZtkCHRiiGiqIQywWOulqkHoiXsFhuXtUHHlqDMwImAQcklLJuNWRczighAZkOypIimhtYpdVVNvbMuTbUqnWIfXJjjIrLXtYjhWVIaduYEAocuueJWDcdMdXwovoYsPAaiRplrSMaPmhoFNTqbOdARwLeYFNPgeXJpKBxmFifZiBrbpceCptReSQNjLMoPolRxEWkwzBbiTLozdWfkxXhqIxUMLNAHSTcZCkqTSKhvzxIBTQgQBtFwuTpghxTtukbhfOJdxtieDttRHEwzUdQiLqlZqRgdkbDSAUeRjLLyBNiTOKxZiaBPVLBHyshNlEoXbEVpbIfsmkUXJSceKhhPLwNBENNHnyvyPPQqfLnfnPrsGnSAGlbxUjtcunXeyjIOGlSrqwlTQOOLlZrvwmXRyyOWbxDXeEZzIQgFUsypPmVSTyHmXgQkjpjyNtOVZIaslBNfNkIwCUisBmjJCbbjMRSuuSujHDxVZebUtQJVrVgkDpOUSOaiuWUsAwTSRtWKTtlJCvxTwyFeuYuajzCeIKdpQRrkXEPclZmnIvmRbQKPUmTnrUhnzJpTEYlptNmHximERosEbfHaWJmTdJbMEBkxIvXeoyxAwpBEjetdRiuhYYnZWUKVccUGxNeylHvsdORYDqJTdcTYPJrAkQGaVQxhdCYhziAcVFtqFJqtfzkxsQoMiSBPeXZKTqAUESRNNUMJFNOYvniCHZQVnNjVuypqlLlRoYGYCvJaIRiJqiehbsblYklZgVycdczYRvrgXQLWXMZDEOqliErVKhejmOhJoFduxsOXOAAUQXmVzFahLnympZApolyzBeXwawJkvlfPjTDWwzvUJMJgwsHkuEFiIVjcrIHexVgwcBdFwLWBKJiZzgqGvnVCSOjAeaSFaipyxqxgXaarqPRTfqxEpGFJylWbleNWGXILQrFPgJwJyrrOYOWOzmufLqfyFKmVKkHyCUepRACMmQXoOhlAXlZdpyASmlxIJwEsEKoVTOCQASKOBvYixmTSlsiuQWwcffqhAHNmmKYBTfJJxBruhjRFGaRZWFstFWKrNjScpPxbVvMhgBKcNSOSSzzvPYAKyHTiMGjHYurnYTbGPVdEGczStuibGZiPZnwrtiNvHrbZTyCtsSYolllPgsEiITdwHoZJtoanQQKixUuIIyeETGODPkBLOsfWczXgkkQtWPgmxhQciWZdBCBSoKvlOdsRcmsHhFtyZeFxJHckOINcYmtpHnxzljphjWSFkWoutleQUxwwlDWSZUVvKYgKshCdiJhVxfRLOdEaZfMNLzUtbyvplDrpudIGJMuuhnxnWQGPIGOadsqXaETguIlYlIRLyMyZCIXKWyNFeAHfVugvheAUUQMNKlPKdqbsnAaZHJrebRuFtlVoflxkZjEHDggCPQbEBPnplJdPTFEYaMwUAlHIaXJaPsJwLuVLYTpLyLnSKzkvhvqNviQwPpTZAYwpZsdkKaWxKljBXzBSUOhNKByydOaXwUrFqFrJtfeMZiCzoxmZQzDOEvycydoNtEFkhSUscSOkSWAVPmBnfvUSuZQtazTPYBPKgeIRHExqWHXvgarqiHMBkijjLHRhDPNGYhNjpFLFXHirTbPpRFxwVZYHtUUFveExLSEnYbDCyjybsbFnIOttyQNXOBuHXBmzohMvLscBTXzUTTYwjQmEosjRmBmeMEEAspthCeWtrGrmbNpTJkAQxYqkOUvHDUSBapsXYIbgksUbxVbGMIeeXbZvSkhbpooBcdMisZzffTSXjZZPyYAhUeHyMoPKLnDmXKlvfFitPhQwdWwDstASLHEMpqzuEoSbuGKQHsYiMuwzkXWjNEJzySoaxVoKwvvKJGWTTGHtbyUkjLMZPacAskyjoOcrZPhbkFzpHbDgrTjBpTfyFRqlwfwJPMAvGmJjXpTvVsdBapiTkuzMVbpNtLdLjnFWpnsthYEHhSjmIDFYybvWaGTsKBywOOspERBajILOdHHECkyHNfqNYWbkUzXXOEGFVNmVUbegQdyuJebShRTbrxJKiYEAKeZjbaYZqeDAcvQOMLrsAUEZvENOLYCJmofvDFvwUXpRfkRVzIEgcZfpammUEDIxDqjwHVeZIVsXyRxWkqYheiMwAXWdHqCsuDbioCpTOhJjDiBopisNhzEsCtOpNyWRzvUBaIPwgHdPBbMTVjagpLpjqjJgVkspdcKJGyUVCeeTjXBAmodIyheQojfidLuMlLxUiDAcPOtSiKmrDJtUqJWsDgjldrTltXrkQTZBOBnhxliaTYITQMguYiFyOTAhKicOyJfRKChfbjpbIYjhxkUrZguEzESXADZvuHoruXJfPJHmiAbmWIFqcJwDNqAWtHYSVfJXzWUNQXgXuymNeaRexHYZvbfeteIOlGCUXfNPAUKQDoMvkauGQKHECMqzlcsfMbvaIDrqdKXMVcwhdhuEEYJhvLyXsGTQVhYcXRcBsOppKSHvBUhwXHcMCnqneNUownmbwTQrqhbmsZjRgwauHwyFzceEKLCqHLTzXGHUhtXMDjiUMjFanxjgwwQPiCGmOmtxaXXHBQRMcdEOnEDwxCkOMMXezwmTZsKRjGJAhIngIMGOStsBqgiKEYSpyWafOyvKgQyrFuzxFVvXzoTudjFMcWwBwipvYJJjjjQrLZWvYhqNtuZmqLsBVeIThlRbmahtXsBUeVlaSDtyMpiLlxKZpqfJpqWPWzHJBOVYyXyFRxyTeaLTsyWjELVviGsxgVjTWjEIJOaFuspRApKCxTCwLlBmeiKifBbyWAjFMOIqKbgoPvKPJwFSATsRegwgWKYTrdmcpRvIpkHXviEaVtaJaRQolgYZlajuniGhmFzndfnSkCMZCiLWBTdOxJbNDKgUmQFxQETJBdJXnoZquRJZkNmgNWmdmOXpzWfCubsfreKvlhOYmzQwXVmiFjDCQEzqbxXLcFsXOqZIAZCvUoYWgMWnDFZkqJRFtwpnWWmOpeXQxFybWUTunWvIEnwvsYNzleidKNPATlAxLhJRCcNWMKLsoWUGeePHfxazwIfnGRVBZkORCNkMuoSzKtPHTiXlTeZGCRTrhtwmHZhffMrfTDoNhbxRiUTbqRjfkyHbJsAfWBmQGHlGsxXwzcfGrjLKkHrqHXJmeMzPADGgNTtbqYPIgQvvPiqcDMyewotMxvPhFKiNxBVyQovyrGGWIZOkWQznSnoYgNThnjmVyrVZRmRvIpLHZYyVxMwclANlnwUaBBSckeJBTDnUcaWCPZcSrSvYcbOgODuBAbkCLltjGqEFBtYwdhVjdXpPIapPDuvMJVbXqHYaSWkdfLLZfRElIJtDagUzyysIdsSzpivtWbWxKbEthaCFkaMfgYtSmGPhEeLGzhfBjclYbUJVImvIuNBqupGkNnhaROTaoxhBelGITNFBJUHnKiEaCBPyJsXxyvpHpAvLLpkJXwFrZRoTbWYVBsGMlPdwlEooOzOmmkMmlZaBpcsBSYxMEqPcMHlENRehZKklOxrQLGuCdviQTinbkPZauLlvsufmhbEvKBoXFWwCOqmZqbcNYgWmHjvOQvJxZVtaRZeeKgenosQZZkgkGIpFjwyVeROKezTliOIfeAIuKkUSDmdlPOSAEhceyffwBBerdqgcmtOTTHJvJsgosOIcqicSRKmuHzLFMbzsYCFWugaGyyzcHUdzmxrbukodchIBkLwAXGKAgMtpFSMLOZlflQcCzAudoWhUZwAwACBPDbmgTVzoqeKXrrTugJOvXMremKDhnnNvUXThngiurKZdDyNNFTfjPBHFSBnhoHuFHDCQfvbJGpsJsrWDpWqVdxDPwyoWwqgqCHPxbfNOcJCiceqXNHPEyiyRIgyUnOrtljubUqPEcCBMclaCCjKWjdojKcWiRhAmJFwqFGYLAIUWgBazAWuvLrcXIqsusJNboGhkNTaRThOHWtUjPnMmmqsRBWJqtulNqhGnBigRjhxfWpcxlfUCiuRZDHCuxoBJEupenPthiznYFyWlRLEfPoKAdWSxCIeRPQJeAgasxKzQhFPOffyCphdttJWnhKFiwNMZaJGVTwSYOmUnzGsuSezcOWAaDAscHriBJYeoWrffVQsKZCyXxhJjxhDcfbzMSECTHKxaiOONERpiUzeCmFEJEivkRZokUAgxxynuNrerHZTzmUBCXZRJduBlChroHyuHPpJVPaPZaOOafOIljZPSjAXCMOjamdUrBxyrxlmaohwmrjlHBreabIfBQivIzsSkxrdDdrGeKYebZWvaVxsTXKQqEnhOaIpIUpuSwytEFNzoiAlUEpvTnJSzJTLyOsUvNUYlFHtmhqdyAtmZXhhaAUGjchHcXhNdjBPmybveIXKqmrVaafKaiyPgbSoqIUiVZUlJHThKFvUxgqVmPMUctScvaqObBAOkxMFErrkWhKYMPDhMocPXgRhBeKDyLhttRsjYLtcKuZoHGGTMoazmGmIMHXDmcrsbLHhllcZtuOIFqdmvOFyvypYHBBRwYjMsbpTJQVolooXicKaqwUwbtRkqZlCyKBrLyLdqDFLLQULryLVFieusTEKUlBmvyyMKrctEKFdgTMXRrXdEbPhWAgAPaUPzDAYQVfUTToJmQSlPsWoPPYehcMWfgOKxEvoKFhCuKdemUwhrHAHQPqISoPtHnJjkdvuMiZXhdUuRhGicAAQTfgHdLQnDJlBcVJnBOBBwbUUowbMmfcqEYvHsRgRQkdikGvirYWbTEkfFTpoNYCZaKknnIoVblmqDxrTnmUomKlIEtyGQRqLYmraefzUUXYkHhQgFuTGIPxcmHOZNYgbfPWNiIGtEACgZHJRYiQhaCZaPPJwBwtzDeQmckIAGiCHoRXaFqwKtOHLMAQgWZvqBEdxrNsyZtTqwShaRswMUViAaYanFBveCGROwdjkhkMebzLuZAptCEVHdpkmIxUJvSlNnDoGoNErzxBVFBykfACEsnzyCwaIhCFhBuCxkjhPjqRWxfVOzmYQkvGSPoPbsqzWlITbYfhEdCLRFDWFsDoxbpsGsKCSKhZxGRqvFCBQheqNktRvkMCHbfGZluULygxCydHOHmhuAAcIdLteLQHucmtQZbgYGJkgAmTeSpDfXMucwWfoCmwUZuKukJhKhdXcZORSloresQJTOrpPNUfElITZGMOqIPYkiTxTBzlUWzGPmbQpLquWWyJIBPHiRlCpJireSIaCRdbDNXqNPAtuqgeUJJKunezzfWmUYyPRgqmlRejXbCMDhVAbtaRuTCugQLOSteDBIARPqDHmqIIEfcjAIwFVzYKQarSmsDamKDRqgfCIynLrnrTDOyqFOpHpzSxDBGHExjnqjGqYEemADvNeyIPlavdlJprNRBFcClYxvetcOvVeMQJXIqRMZoSydxdHPDCjIvudjutqinpbCicZJjFbniMWTUIkSjwoOjzsWuvUtCOsPdoRqamDHFGOwnlWthnwMOuSJgVninFMtovKFXziSLutlgFJecObZeyyzLmoICEZaFkCWFMBDQjfOvnyflVdKYAPWmaPWYsjvCGUrmvBzuxtNPnMfxcSvwOVgXJVArrgalLebnGEAtVwFhsNuBcXeOKOyXdxjWHcaCUWLYsiWTvijAKtjxMerltMACeCOXYfFqngAuCzaVxNoCdygHeijjmfkObiljuYgkeJEYYGlziRWXmKDCPPhbBloDLHXcvBRmMdCGMomOQTVSXncOgDAjDrJWYIDezbbRqezdMwfxumAoiKhojQeTunqhsCzNGnWUFjtjmYgSmcnLFxLxIOsSLAcEQYFGTqvunGCCEAaZiszsdKtegBYyvCyWstnkfVggVBwDUEoFGAZfJQhZPWwkcSAVyHLlKPncoRJywSdRthuxvSBxJqWSfMRCIoyinxQugSDYDjZNOeYUWMOGwQgZNbHEFbdFrfsOiVkcTTEhLHQjqqPGCAYOsVvRVGqmLtZUcfWxqXSvcrYpRFkKGXvWbjnHYbzRZhAnwNGFaRvTDkesEoRdpbCOGaduBgSUqoEiWLMXuMlGAAfjhWEOMVbhgTatWdkwMKzFSBUstONdSqWxsIgdZdpwuSPTeVeKUrPJTZuaPtkWfnEVhSgNmdzrjiLAslpLYWnyeRVtvEDSKfRbIDFmyfjOaiMdFTlMiwWalumutrhFEIkIIBZfyrChsHsPyNxFDDlarabeutOgKqOhMfpXzKdPbDuCGTVOAlegIIuNZCeZvZInXsXqOqYYLhwIURyZKyxAnzJtekDLhkpMiOCPmAUiitYmSOUHUqZVgOkESwqvIbefofPFxAkiVXusXXSmhPGRLPwvPDYalpNsajmiQQggNafYkYFZBtMvHmqgfRuvzUeabBlTyQPrUmlcfwWhdQfIBdbnjlwwvDIVryJFqNklFzzUJELIUxwXtcgcHFJdGdswvuxlVFqCBLFVxMBlicMwofeufPqOUGWPYHkxSDlynNcgxsemOWnXsLNorSeBCzVMetDitlTiyQTjUPVQGbJbFHeOQztOKBPvHTMgUTKXVmtWeHWfpzeoQyzlWsJHWgtWDDStOoszjyUzesXcKuzzBEBeaJYSDTEOsTInqrHOkUUBQRgmHdcggrnSRPMeqrIPtTZXetjFdjYUaFNdjULjMNdQinHBGOiQVXMAVVIqnraOcyXDulAVGuqOyurYTHxJjLmGuZeaOtCsefrwuuXZPPavtRJcenkopjcbpkPHcBpCZdZWbNTHqQbrmSFNeDufzaVESWiltPDLtnPsnAMzWXgxtbtAKYEyTYLoGZLMqFarlgXaNTwTkaDQHGmnLFROFILhPEBQmGwVJrFvCfmzojIiHRbDJHoyrafhoarkkzMXTjSwAMwLBIHeIBeSCjrdmdZhDriWhpujtPiEdbJQwysXkZUyjPUMxvDjGHkcFydLybAJkRyNsHPALGHBcjvkNCFkjzQduAqykOXcormVQOzfzyHFHlyhYnnQVRajlAqCUvJwPVoozFzCXCuIJmgUwvNqTFsCGCVdrqgrSAmCIuEvWWJsvhObTPvDankGadecSCEgYicBjFaKoZKPNmqABbmZFloQqaOlbAeQdbRyDZkGSYmumEmxxIlTcLYofDGpSXGrWnnVzqhtQNIzFgxenIjXMZSNPTZPUieTgXfkTirdSxpvcIeSErgXMwQDusvEUcOPoVTsuiIrrEjdeILXSMDDswkskqqaRtsvxAiAhxnWnFriCfpbhEYccKFKUleGRRJyfrThmlVnSIfbjAUkQQAMSobRiJiEoijDEdqcFSDXLsClWbBBCVqLQEHygvNSrvrDYZxuTEeoVBVsfVYdOGBLFOKIzNtVjGajUqhYBXdDfxBhNRDrhDAlGeSsTdmYsMTSVZIQApjXCXMPgvvbwdYRGPiGvHeXMJoLdPktllTQrfHygCDnVVzfcYcKFSxgteFknMdwnYVQxEgbPeZOxNDDCCyDHDjHUTepHsjVJfmflGqGAptCKoTudNSpaAdetirWqrJjQgwyFFmDUVrPprWygSQJrUcVCOcIWGEVPUcmiuYDDrXNpwlXgSLqkUgUkkipeLyjyhgAARvBRHHhBRibOabdETRFeBkvudMqBMznzGYNgNatqrSAKjLQpdaPVYyAYoEHVYAhWBOdKqJjxZEYxJRUojpAKJuavBFfqEaAMyyaCfbrEvvDvIuTjrPJUPPhoaLeFGCjRvtSDiYRAoPpftfSDbybhrcEKdjaFSkwMhsOrLgFEaVExWnufoNMZNsyMfGwQXdgOkKPgaurDpnFJmxhtbmlXuZkoeXyyVWXqhoQrSJBMViFjtSvWEYTnAalMGJtdCFqgLKZEcfwtfUjBBkXeQETxfjaBRGSbXZehpjUFCOJqJHKWFdHWeSRaYtRorBplRHLzLvFfqyLpPeFSZfEGWRmcnkDVBRKDlXQtWWklhSLnAdZVSURIytxmpAGIxUOHOrAgboztbdOvpDznDvowAKcieYGeBECpdSTOpxskIbZqWdDdUQgmlbrLXuIuHLOMahLlVFkOPGZVExVYtaJIXlkVGAHXOSCYloJFPfNKDsDOaTFTaqRGAQhyOLaKVPWCqfekurKmxoWdTLwsBiTyPBTGwLDWwSjKwbXhGuZqKzELnFfxkvKRsZQnwtDBLeaivItjHEAiGAeQcTTpCaKKBNPvVFaYoAehFnpMLNYjowaHGakXWuhZJiHHnlATLYxwOXgMHGsxvILsCznBPRZMhHvsoLVHQhadVfbemXVVkkdlTOzvubqocIaicBJwrMEEFkxjyfHEHdaDoDJGwGvcJWhzrsPJYkrawsayklRzXkdDYkLAEJSWyojlKIzcUkKttPGqOBCvXveEpcajvEFSrnCORPiqawCZXyfFBvCaNFfklUgAgPfJbWOJuWLPhauLFqQqcdWQCZvIWphKIKTmQlYIAiPuiWzWTiTMropStBeNmYJESSiwNamZrAHevCRCXPlcIKKwvyXnClQYuAyzhTbKGAEIuWqjPdvBGwUspEzizkqArSJTrMhcUmaEXuFckFryVwtPWnsDNbMpAYDaFvMrtyyCfCfFSaVZAruIntKocCTKFvbRGrBAPGugAOzmGdTwSuVfPwpAOhuRPWjLDYeyUQQWRnpqTIIZdzkehtqmgKEraVmSrekIShtijDQvOiBkrqSCDwJQzFMQIWuuuLKdvAvgJgBGUrvYaVdsYnSjUHeMDSevHmWvMcKPaRTbjGhFaMbWhELvbYFSIWuUWfTTHzKOvXItjsxYCrhXkbLrEVPODdyDYJljuImhdLCnerGmqUauPDBflQpvcWCZVihazAOEUPWaGQNJEqPqNWbElSibuUbcQJsjadSyNCipqVZpQggsdODomYEKZmWuVFSIKzkZNYQAzDoQgOMAiOtYAKpldyKIQgmjckJkmDiPzEUAmFttINMrDmngzxXInxfvstVSEHGhFzlQpOCHUmSYdaFXylHpoAliYGdIchAMHNKTKKjiNCAlwpuxYBiCCeKkIBOOLDSnppUSwcgAdyBewdeXGTxfYbpUNegepRDveGVEsetFPZDHnmjTDEEqTyuhcCMrHKQKlEVtfQUQArNciDRfdbJDXDCnOdRJvtQPCIPmEswBKEvMuXVTVumKiMdpunlMqXZOjxAajhUstmKWypqDzkTyMKADgUhleFbISiYWaNNNlxUzjUMuKCCTORrkkAAvVhXYWgPaLfWOShmprTCasDZmxnHbqvnQDbbtuYPpaozTPbMbDJdDFOExJnIgLkdzOTYJxpnjXcwEEpsyrWuQFCYpVmUSDCNdAAUgnMnXyiQnWuGtozxgFnbxMjWwOqGPczpffDuNzUAvJJbfXQkAxKHelkglMoGQlVDBCKiImEcCJpOAslAixQuCeutYFjUpaIYrULPjOwBOuiwvfWiqJOLaBKMzdRnpggrxyxJypGMBRNHejoWaHmVNbAFhPIcRoKNpPxqplVFlNTNFxdwkOpLrWGSBfZjQoQqcUkfCvvRKhRDqYoygKYEyaBPAixWoJpsJUfaFuUtOmuskYMmtLqsZhftpDjMmwBIrMZxQonwXHVgDBaTpJBIlbcEsPyiXzcuDljKpukmpRnnCEfcglmFMBXVPhSCuMlFdBzqZReDkUesUNEVmxpBMdaErmOXcfMgePLKqprLTgqbydfYPGjQeydtmrLDIsDfCavGVKNHqOYvwRaRGEhJnyeZuOhezRoAKSMLHShIvJtjOHldfygpxVxLFwLAQtamzCMMmtlFJEFIbGhjuQoyiusGHgpVAacazsWLCOGoVXoGgwMBjAxaUtZGGeYYlRktfnzjbfaAPrAxTnwhgsXzFHoTcYDvCEiyqpNbSwhQfPiytzjIMVCZVamKUKbCWrujmUisgxaoRJaxpYMssTZJQxqxEpNEnGZgWjzQGwnDCFIVrxjuxVggWqjyYskgZrQVPKKcsalALusJCNVJFHAkhlnzUUziLPDmWOjRCKAwMAGkyPIEGndIBiwnsnuyqDvwdjDmdfuIfKPkzpVZBmyHdKthwIPgrOyxPGISKoBmDrIQdmXMgyBcgXmRUvhLXYWwybUNcWtfSwxbgERjhAeFsfygbHdoXGHmALDUgUDYHThcMnoDROrQQmmeXAGAirjqgrXgwIRgHcTAapPEjedAvIJUnPcmMPDzXAaoawYWqextyxAvxdYRERBfcfGmLATlhVPCigLgKCtMCnbvAlFdbOOmcPVprVTABYoOKEeLAMqgIqQGDTwGngZuqUNbDfRQageuSwFyZZSIieiMFXczHDBHqNUOeCqQjTftUMFTLCXrNTsqWQnsGxhrNuTOYBqkpuuChJKRPUBFAczTmEqqyXZnhCZYTtMLCOwnrETJrbrRVxdNLchbLmOWyhsqbdilJAJWdlEznrmaTCrCDbhnTfBzmRbVzYGLEZxzHcSOIOaClHoHKAVeXbgSxUkJnXqwMxKrdPvbNXrKkbPlsKNqQPXZDcgjEjszGsSUGZJgLcAUAaUZbEBsbKlrnNVMKrgDKNGcKqozxYunOOHRbGdoZGsxvntDKXRYwJqKjmtfypPVTawyHpgKVaCaupsTfFpeRuPnpowJYBVajcHEKGibiXMLNdCqnvpAIhEvIVqddLZQCkMDKWoxPCQWKutRUMXqjWwjvYHUBkxWzxtHajnyxqttFMeJGXaIndYcKNVhzErkhhfWGevdxMhMRKoageGKtRxAaabIzvUKwSXgSUJHxHBBRHNURumMbEfEKNgLeFCCEwnuBNdzOXFYYsUCCOYcDNqHLNWrRcjeaDglYJfeNOYbYyRxlJIzgxPmRkLHwKOgZGXKNJQOVVOxqXdvFqIpBYSnuhGscpEQGwuURBYciybHsRXTimebWCfZJtqkdJlekvSyRCtHBGPJHEMVwXVPKXjfvJeXVXtYUNcYYkLqVTVjQXlwqfqWAWlnnETOcTjtbwlquVnQkdVOGFwGWPoXEMQbTGTDWAdQCLxGfqajXHTAEwHvRjKRMkHlDbafmiuYuhEIMvViuYnRURXWDuhTTYcDgdnNHsSDarQYjqWumKHNTpPcACIdaEtWmGrWtAPQXGhIdcLNuxxGqWnrmpGjoMdMSCPOCUmRQutbpRfHlQqsSngWGMQPGgSaUSvbLsJeJmwNRZrILlCqdnZcnxFxYMoOjYfCmUUTZBhlmCQbxeTwOlTXlrmdiSdZnnnAuJhfiyMKFbXtmqysmKfKLHZSmCUxexJRIwcpsQCAZvogXhiXESzuSvERXQiGXYJHvMoPUynlcqfelRMtOxsbECHBSxAwKQCcjTFtpQfomNqQKifgDNrWUSbQJUYlGVdtTieCGtbdqIeZOeceCBhgJAlgRZcRodQAaijtQZwnDjosphUKjMXlJplRXnZEnFiOukLMkddzHGsulhNFpIoGjabhOjpfqLFeJccoMqACNMBZizdyeweaGagGxecnGsbhuvLaeGLmJwlIgGaZsTVQQluCWZKtfLKOSLfQNZlaAekrVxuzCBdcZERbTxhKMsAGQjcWsSHzJUmPHnSWkYfQNzZtUNopzUJmxGHXqEGkftylZSqxjhzSrPaymPgsGOigXBGsLhtxOdbAOhAxbGOvanaWYYEPikWodjCUTfVaDuOKyWkGkmoUAsGkLGILpnvllTrYbouOnavlofKBgDrNdxOBjGwXyhSTsxAmOrTlypiCEVZyxziQajbrRWXyOwcLMJTxVZqQldmssSmsqxOuSWKoiJJidMSqJHCfuLDJPGoLVSfzmvHQRfuNtVhuahDwyeCKgWVyYZfyxxGXCdQhLfgSLOCkOlUylogzKjCITwiCOXAQpiDnIivlQgIdzSjAIgTHOLqvudHVEOqcqYEhHRTyfPUUkzLJysfqZNXKGdLWrbubJGAKrSbKnZworwzfjGYtPzqnVkSgrBacdkDyLNqtQXfxFUHsCEIlPbPkoEzwvpdDFrvuhlOdduflZDpdifUkukyUXtWBmCizJVERZhAXoXQngmcYjhzeNFWmZFPKlaPNUrzbGpBhPvmcWjPZQcsNpcYunzQvLLieeJULkBFAVKFLMPmohzcMRkTHReHnhYkasbyDVczblLeocNljlxFKhjZwiBBMLOxkSmnlwXqtbCNTiUppQHkNHpMmAIHOwOsIwIVyixejEjOgQBtIbMlaXmolMORDPwyBlvXDQSzcXcDqZvbuIjxNTMYgqxZKxFNsxMsjkunLVgBDjnbMzYOvJhBRTPlgfjJXMKuQFoAmSCaLEpZpZXgELJTunlLkdifGzajwIzDrMXveyopWFgxmbRyYpdlCZhpzjUIgaqSSnICTtzwlRXSzasfxQrYSkgppvbmbkyCZuKkCilJcYhDZxzHTMFMjetAjomsFtiKyKQXJNSvWlTbZiAPqVLcNxRJIpqLoYPXuqBECdRwSNebmtLzuhyruiLFrlCigihdMDMcdAnmrJhqwWrhCqJpJfmNZffkZaUelIflGxcrIQtsPuPyKeBhpYZxmnibRJCMAqnDbBziuvlRGOUoxYsUCANJmPsPLiPBYUDgMHKeGTBihGNrAqHmGdCLjkwNmIgoGzJEgnrOIupuRztQAXmQcpxMLNKhnQAeoENjpTRxnZZJEyEnUpUlaCsXqZrLCFqQYfzOXJQmqwwdphCnTIQAYYHBrmFsWAAyMavgQVRcVbzYocbzOBvCwtXWPZreVwqeGXWIxTMlckaITKCefRqpiDScODWKykSQkAazoFtbHsJEutIbSquWMqDshoNcLmByrFfEyRNgWHrhRbRTWcQvVLWPyTmcJmYUGXOpSGxBWEesFmYzHDpjDXgeDqgtddotnOjpxhkWDgTIYlDVgFWCTNdbbYBIooyyIkyIgxFbJXdlIUztGTJwEPtBpMcwNXXhVvWrHwogseBgKKQXHxdvCatOVrqutUVOqnhjCXTrTIracmmUWlwHujQCEbeHkfggZsNNpBqBNNNQmtZPtMEFKyVJrpridABZVlmhQcYfxLRzlVJeiGJmzQxBzHETxJJSUciwDDAlhGArEgkVrYhELubVYAypjQFLEPzXbuyLKFlvSPygHbCNMFBaHvAKdewlcsPdHzyFtOCxWEBCitSAiAkGUnwgDhAWmRcTJBqqrqkQhVzXFsEBoFmmMMvRJhBzKQvWqAYverNnFFnebcUCduSxNnFOWUfdOFBsMScTlRTFvBrkraNdjRCTHNlzfqkBGlhDaIcwblcrISirCNZDbWzjZdCRhZykCajBkSowJHHWDQMAHROVifHaCiYbZSmAkwseYZKBWGQYfnHLMikNOpwAjLlMdxroCjcrGyQacdTdrhtnYaJIicmZoQuKqSQVIvhNNxIoJUVJqOTVOYDXcafJQUCWeyWradeBXEWrEofbgOOCWhVZcaXiYYJMYcoikNFTZzWjXiAhwXwDFbRplVitEySnlBPYjXjuUwxmeMxiyocIubKDEtATNTHUsYevNekSAaUGObBZxDWyQnJNyWXQStuotgwuQFoKbkFJAsUsJKhzGnFkyZDEMNCICeVChGRsMjgRsXqJwKFjLIXeEwUWijxclkFcxUfKiqblvPIFKxKFIMlpJfExguzBeTPSMwRnnHdYHrPnvWxlHlXifKjvCapljEHlmjtSKcLYpiLhvGGHedVUKSSVyJntvgugduoidKKWWSpsFhtGSqNXIBAiTZRtcRbinrlgnpjDJpThbPbYxsZiDcVuBfCzkAPWggYAhRGyIGiPBwOulhuzteItVTHiGjYvCfbkuFqSyJTNRSTssUUYFHCgFXyJTQrEeOiKNmZfvWSEpsrPvJPgkyPznUPmYvhLmdwxNLPLOGDlfVIWocDlefwpZUtpaKWbyZGAWrdNRGViTPassZczXOXXCERAKXlqWYJItUvAeElDemhZhuYqZzKqtszgNxlhzjTJJICarvwWAVAbebckmdNGaafWXsrPaXGSaVXhFfzHGMLDpHrlHQAGTJFLVJGYvYitneaoEFCknAfvXdZolVshHLacqopwvQbZdSvMYERkfYjmpoKzSKSQxuZOvPUGRvrDEPrUiGmEifTDxVXHGsMhjNngZuYbHIWnbdOTUCvhGnevtlMKFIECjtgsLkeJUrkKulohvRbswelZobnQfBClSlKYRATaNzFATOIYAIvnlXrdqnabdZISETFWRyXkautVzxOdZNnZydhCgxnsCScxQkgVEsSLMWTOttouXOjTHdJvJEZNJzRfMuJYbAfFhYiZEeEMwcDoDfrvOnNtbnugLPwwfGbKqYPqCNnNVekQqWzENJTPGNflEvRugziyPslpTmFTDNoCwcvWPLfGEetdfiaFldYkxlzYAfhyCDzUwQltdQsxMmODoRAdbIBQihKSxjpFloatXxavzsRpDzFsBHtBUuBKrLmrMkLCwQksEvQlykpQvuTuApfLNZRjxIYzTRhBCLlvHlBOftoqiHKPeJDnQrobHerqQffFWLpsvMCcswkwOQRaljIqnFzzJEEtUcOJfjDufqcaosMXcYUFTtggMSDxbPCdtmJruXluOsTiECXqCkVsjtrgLsYLTiTscNzmiaaPtILgtvxFFtmrDHtEqQLxICDKAqzpoesswwrGiwHUiLgWoENkSWLBrYaCVKTsMJKtzexLFSXRjfrHojrWOZgpzRVaFgjOKqAVldgvIdCGXFbNnPSkmdTfSzVjFAgYfsMVBxEXbctfXMmvEKxcFOfTrqRbUYTwdjsrYWyOVJjZDVRGGbitrsNllhCCWNhmmYSYYNmoRRafLcizCmLAQwXRjZiVrAvpxMSqHspvyBGzvUGLzjFwqHXOnQknpqrgrwOsBlGRigVLzDKaNiEvsNWATcxfwYOOTxcSvowBGSTzyAmofAfRZOsYdcUkvdpPnhnPxmNhNedrvsAflpliSkmlEvwwjjeXpveEwEhuaOcBRzHzYkNqbeOjuQQkrtCjZQMmzWseppSqLLkVwYiFjybTRIyNWjUhgPqmgxUkELqvcRAluyPcGLQEzeCpKePEQsWSExcWONMBnOWDkKjRpZeQRpBLSXXyYaImXMndHGzikezHRkanuOxxZXakBBfMIQTNkghSubxyvVnrMObFGwsEqoVzMXBabMlGoDnZsEnbPoCUWtEIqJexzSfRGLNDdbOBZkxHpGUiBpIMYOPEIwfYZDSoflGIHgJYeBihTlvwdlRnnQbQddPpqTkZkThAgHRObbmkBUsiItVnvgDQiHKBBHTDPtGUniBWiRPKqzSMTfBGYJhJMQsHUUmDpjoHlFpEHdyXIznxyNVyJNzJnUSvbJKoCYdjzRIgYPVJVjmpLHjifNGmOZOqwWmdVWPMviQSSdciZlYRsjuslEsWmlqIMBjrBzRwoCHZVozlqdbytJNZzlOjMzXITvitQfrXPfWkkeHWaooGLttEiksogjYkoKkJsDgmeGofvsMqpStBKhIiITCFjIsSvTAlGyZiwUShRJGHlEYcOdFVBMUaOZNUwlHZCeuDWOKIKDtNRMdkYhoOiJYaUQIgtPVgmoShIxSKcoRBTzSzZJYALLhCKVznIXjXactIAGvxSeusTtGYjAoQLZVCiMTgFoZLSkIcaINrUNUSQQuxxcXRJyFrLKZUxfMPmnsBPFdBlojWyMqXLVMAjHvyiLXCbgUPzFkCcQuFanNUbFUzLBCOedrGMckJBdAjHvWBquoHckUeZrOfVDGTmlmkjzuiSQtidiPofSEUrQBLweqsteNnqSFbqswvTYkEfbAiEbecbRsmUpyTLDdCVPTqLoILuIkhihVwDQmcDEjTbqGuGwsWZoUBtNruyDAPjBMajNSMuRBJsjPhWkuRbPLEsyNCmNSjdzHlTccHwINFJzoKVSXMOOyjlrFBavTxFbfkclCJvhBjxGqtffMtjeNsDaYiCzEGujkTsOFtMCuPeAawAiPooifIjQrndtIyhacKuHglRvLOrKTXokXrqCWWusITegIoAqoNKrVALGasqfZUFADEsTSVlGjaAeRWpszOUGxacFOwGZEtXXvuvmekHzFIuWrJWHjiUDLpPWhroaAcwXNPvxEZszvmcGJTnyKiYTcYmGrbJOzBGDITXFNyHhOQtwbowTbKbJieqcgMfyVbnZmDBiVstAKkPPFNXnKKLhCwcSTrkkyQevmcvuMEdIrYmXdiZtfEAMcufXyOnooDgPDgoJhYCtuMcHikLVEzkUusGzfPqrawmgeFKyAqrKbQdlCuwppnIbGEwcmOzaHCUYPfXFJNwjVGSpFrQpvVRANfAJdjzCCTtCPiFZuDObUbSnbpFkdXXpklefyWikyDGUGsZpPhfXwClBPWixrbpIqDZntadehkPtOUdPwpXrQBoXgskzLMXqBUETEFCItPDHdmUXeWdHPkfVPyPIkibzsPMkTfJCcsNcBlgnUjMXCrwRYUUAWlwtKwqyRByAYwJRKhOhKmrtWpIBxsAJNefTcqRczpBRpnkTrOilaHiLUzcSjkGnMjZknSkxtWtJflexGYiPFwBlcVhodkAnebQwCHtBmNFgaTEMAEUcHhVAELMttYfQjFswmtpgNPPvtxgGlQkwwkQuRPczmwDhShtONHQpLJpNScXXplUvKhQIavqvnaiBwvqzTFXfmgQqdxcbalVXhyWOnVsUnDiQppLFOSUdUGtujzjxBGGYbilQkPoJhlQaOiNydYbYMcVidpqyEeHClEXBDWowRmjjFJxSKqJOlLjKBZKVCyZjUztNicMrigbonwqwbpPmtfOndlbUQiOTKEHaAnhpUqzhrDcOkKQNLJUIpTArCZXiHrRASTPHcGphfpanTnFMigpAWMqWGLLQvoeyLgFyZSqBrthLOZSAmxbYEozyHXnocKpEvlpHBhYvkmFkDqLUMwsISKFuTNnvWhsUsgTScdGqZlvrYjmUrUhvrGVfHpQwGpYlBDPKLjsPIrwPlUGKUtUfzrbedSOJGOginOZwNmTDgDfptKFLhkDljMXosQhYdMRqGuYIxKDbyxtqWMvwhUhhiStAPcZwhwoEYEEzHccDTHQDAHLwvszpMPceWeZOJzoATzmBUZyuHlxmvYFsYEdnTmloGoRlMUvtugBanKzrORZkJOTXvNlouoerEfrBlsPladQBNdnByeonYhKMkYweYikWtapMFWSUtAUikTCiWwDltWuahETHhvXskBZxFJThkpduKUulaVIvTXUTkdvWornuZqqfoursbBdgubZYiEJeALgnGzLCccNOYERHxtXQFuuAWZgEnawkNSDHUMpgsVFdEPKJInUMNMIYrNtimTTLMFPPjRakcPBeoRUVyhGFaetUAGJpbHzilISznNjhplowMCyHMnLNhKNIlUYvhYCKUlJqGyRuQQUoemYwLgyLiVQteTqmsTQtTMgVUgBFnSEexIluuLymiuWxJnjRmnOrCTECzzKjlrsaypXYxTltvRXVlKsetejZxBkpHXsCeuOJlToeJQShsvriIkCXQsNefZbNxxmQrqkJPrgWnAzftgSaYVMQsYZNfVjXXhqEzyQuNyLTCICklbWaYZSIUniiIruwadALhsRcdcmkBRidYJfVZTRigDYbonuJjqimXAeZQJRbUYeeutmViVwLWXZHeyZMRfoniglLgTGGExWtNrTjfUppRqdEpcaoLvxavYwIhlNXpRHrHrRCWmnrHUugGjemMJfNCEdQnDWoFqCXbaFVTvPnPeaRDJNjWAmXMAvtRfPpeLhotgEBqXeFbDLAwiqukzixunEhhnSfGXhUVIOCYCPZtlZKjsjVPhUvGnZPPIJgoGZudlTGzMZlxMqdwPEWBInNXDnxLyBvkCKoaASBNLlsKTJmShgOPjeduRRjvSQQibPioWLcTmawvEvyxRiOoGsMeXSKLzXrLeTpagDjyJzjJOHDgaaDLwMUQFKVKtBVSIISGBGJKkmLDoyaOTvqhWfSwRBzbIzflegrfDHQnKoendylhPBokKoaaRZAWwFjwzgOFCItFBCOviLrIaSKfxcAJBqGnwtTuTIjWHFELIJKCjXFSNhtFNMlzGrSQbuXxAucpBFtjdMcUQGMfEDGYdQsknQWengRbCDBEBsQFGnmpKwBZqIUzTMYuDZNgcTCmUCnlabZKHeAqbtQuSLjLaAiDjxqMCGEVOzOUNeOIOqJkUnqoPLrNcpkHUCZvpfJYuZpPTCwwXhXzuxJUIIrZbePJjJyGnJWPdZnBobPcgtSBsexrAiWZnzsOFEmeNGsmZiCNBaQFDlNYstXROTmZXQfPDQVlIJqRrHkmmjdGpYTNAdgtqswlYIUcGpPpkVzvzWNnkNhADEAJVmLJgwjHHYLqvnOPQeQqWnrfkSYXABuPYEEfANdkTCAziXDJhSwLHNTGeyDuycFAtdziYgGlIQZKbsJorNxRTNdqPcseoyAgSGFaOZznJlgWMyVzNdkADHhsGSXxhFNPDBZEnDTzqATiuJsbAqqTpHSjbrOPIfSgTCBnfWTvwlnnNNVCxiJvibyDTBXrptpdOyngrITeZahtVvnRsqixUnNRVUHihFdzCMCeKoSGSPKMbTrlSNNtIthMajLnVBvrWIvgEXrhwfiDnVwnecNdCVRvOnqrfCsGhMraXjBTLpefXnDXlmsBcVmqwNWWxAiQzIjXpCBaynUwjbyrCnagUoFkHzLikCaxjSreeQAcqgvbdGWtZPciGMOHfjyOSlsrKkjAASZwhhhPNFrLNOsTWvppFGLKkRFLaDbXEHPWYuyTIFIhQxBrXbCrSEroRxHpXkhzwTrWzpDuXYVKBSwIFFmkyNFSaniUZSYkClzfDwEKXfXGZGrwSJrjLHYSSffFWjROkLWGyDbPjNHkdouoOptsDvbhCxwhynXbrFNbhxAJRIOYdPdGxYlWFKdhAlqHoolruxcGSfrcvUxdDbsKaGAbNKmWrEmyGibmyQFoUHFJmnFiBTSfAFvYZQCCTSaLvWIwrmRZPJfHLaRnrOxHVyjEJydKeYOENDerUBBccJeUbjeVZglLPRONvFHgichXFovPqupMxtEaefybUQLjnLUvpuIOPvNIxZqzgaamaPQWcKRxPtmYQqRxEssMjSgUMKBGILtpOczcsSwSicHCvokiBCwrjuymGWtxIiTWNDSVCtPURGBHglmzOAvdSFgnwSwmsblSExoovuqhTpjHyozxGqcliwljgCynEaapGidaTyrCajCBLYCzMqmcdwIAPhzWnaUlJjOPXnJoAsdeFWuzSDoluDGUrAcdSVpMhbieQbCbtkWCAstdWPXqWiraWrWgrfmDkXNQwMfAubeqrqZGYhzPRRLesmwssbvSTqCgjvEvOHFOUrygjYyjuAaXqocKWNeNJmiYRoScIdFZaRLiHETQZYYNZBabCsOTYZsKjGFHUEAcjISEYLclqzoqBpyLoOxqiMjBKEAQuSFHXBDByTgALlosMFDoRGKSojFuYaxxMzmszDQfPgtKyIUlmodgkErvAhjICxspZTpInlxamLOXtDrTSrdGXVVpRGBkFZYuaZPxuAdHEaDHZhEYpXUHevrSZkowEMQswnDcWwxZIdTHJoZvddZsxHVgXWjhcUHUxkgIyveSnjxwKdZWyAerGfkArtWmWQWeasAQVyKXnrlSPRLLUxzTFhpKGMgqQTFdsAAfRoeTlntihGJpEYcFjpuNwDUpEGlxFKsUHCCZRtaaQbyyHRGdyjrMRuyFnvVEtehPeNwMeexIqdSGmYFRRcNprrbWrLZInFlPGQVnrSkQDPPPLbGoByAIFqHJQUDiqyoUmOFoiMctCCVTUkiIAJRKIHLXmnHynVKWFJqBkleykXxQbVsNpsRnuelMKeTOILtOqkyfDQILEVmYaKottJgGaVeSswgjopSSLyUcGdUKZVaSDlPaLRGwuXrSBALKxNYxfLEdiEbaVPPSSWvObiayTMZrqljbwkTijJxyBXpqNdKKwGNkKBqfzMvAtoxooiwzgFtAqZVgJOwHvEbBkRwbdmbbixBKwxRUqJHOLvwGROuKScenvgfouEozjiWAGVeTugZyRZyXOuyxoIOIVbwGoNhtwoZugZamIwvpHQbwGDbqsFyAGPfITJROtoVUhmQKeHiUoLpPRlNGfYpxuXPcHShnaXXEihfVIMPAvdSetjWIKCdZuLjuGYUiELGwslPbWqRwaclChpkbBIpaYKVDcTlirxddIddOiwzPOngmGUFzTemUaLYpHPFYARbhDSdOtysocHitVlMYGARRnwFJgcyxWwmvMFlNqnufceUfjXtEPXwmlgiPTYaTlDZnUPRXwAmNhrgPzbrLKSVTgiKvbJjeUzGSUjcMeJIxAGpKmmVHsESAMjJWqdUxEpcCtpgWVUVXFkxVrJBEnRJUAJAQTnhXFUDpTXhjXpQsTHqfNbqwimenwJXtbJOLAexiZepQEataqHEsEaVvINIreLPCuhLiXkhbsmRUDiqCgNogVtrqvWzAvflhzLyfaKPqcgORSHhSdLLveISpblsyxyCCrQjtfpRxQdcvCeggJTfvkWqvLWtSaAQgJHeDfqSyINbNgqvEhMLSJyZpjmoEDdEAXbZqUrOpGHKMjjQLOMLwBXrfncUPOTqIfPUWWPqIhsBNROZQxFsDLpbOjPbeBFKMVgesRWtmhqeXFAdfITjXaQPNUkHZGUnYDTGgZhBsxQuoMGQunwXzenVPLPepPaXfweCFtJzmKaggSHPoJDCPployYFxkHwTkawrsfMZKXIEFtYrWHvbFslgpHLsfrbpIaRxNXJUgTXtWJvRaiVHFzHQqrcnIuMbLnIXCBMoVNzcYhQTMWGcVzBHcSrTRtmFWGUFpYdKeiKPrlqbSVpQWZoDtHkJdSgfCaENYCAfcMfotUzCCeFIBXPtEgiDcwMkNemMfZkIDMCMzpEGEBKUTVyXhnrljHyPTbycefAHJZxaypJvMECeBlBbzhipFdWjqCJwHkQvnIuMeJzQApQhTnjzkDjbPnJEjIowZiHkkXWXspthiinMpNaeOgMPhyDuqbJPiSNMAjztISBpHWWEynyNDKsOKOfyiacJYPbaugRMRvctZvsWeFTNjGtaKDDgntNqzxdFoTwbXDIpKkQyntRulyQPSaEzpEKcWnJzyZBziOnVaWtwfucSRPdkwSWZUEsAPxaGkPoZYpkvCrEYebHUxIKkMuJHqokRmXxzVrHADfyOwRFECfcNquHHKmfdVvVLhVUpIIbKKyRAzlUsProlKiASUQwSZANMRbigfgmlBByVJHksLetEeBZERgYMAcbOJFrFoWjdJSrwPlrlLFBRtrXqSbASWPevvtZGblZEEgSsBOYfyNQeozlLNBbJMyGKfptUWikMaxIUrwAaigkImXvXEmUgwnCDqqHGLxUJBuOgiWUAOdPkKOMwzCXzigUTVeqGPRRqLUPUAQDSPrCTzqDEsFFSUUDrICWsyRSYjrnHDFdXdNWmvouxWcdflZYdqTSkHbxpdQaPmYzayAnwJoYEtgNBWSKYwxeuoOgEDYoKsVttlSYHgVkDfAFGRGZAJPUHLIzpJIDzrbNNHCaqYzLdxHnvOmupfiBYVkGopQOPbDYvQEVdpvCdFcsqXbMrrlVTuDXhiANQbdlwXKyBxGEKhXPHVvtxqgJWqlnCkEiODKEzcUPQQzfwIocaIuIFuQGOJIQpLsYZCizkBSqeTezEaXaFWBVulWNQcuxrkfWDzNOTvIAMteTETcNDlfRjzgBhtuewwtmSjjJpWZWcNnReVRfxyZTpajwoUdOxbMRqOXZxpHCBOhMaCyIpnfGqUvUlOqssGJdohcFOjVPzsXZzEruhBlJrNYLXXbAXAbRHXqrERXrSSoaavysojJZmrvAxgTRSdQIBfPJTRkYdUYvoPEWHvkreWuYjYATddfKsosPAAXCMRYhHGEtyszmJYbgSRboCBCWudKYSBPJfcdIXxlWEFKqTpJsiaEzFTAtmwECzHlfHKdnasDvIxhvXGCHSMydxXoKBnlkqknfKAIUeHYmIKCPlvexQNqCFWeqiAPVndVaZIjyUvkpwUfdFrqlboAPmUeRKnJQlSRAhSbFczbVDSuxGLWvSjrPSFISNmdGakUjoszXydFdyMroyLaeScWJGXtMUFLTzxuBKhcphafheysyKNVaZteTvLfFcZufKRSeahYCbeYySTnpsTeTLTAyJAWqiGHUAhcGEKWmrKhIwOnsQYKXYafQdFMJKCBjCQqwSGfjivUJqwPfcpKyJEGNRuHsTmCAecDcgUTvFVtBwqPDkAMgLOBLBDoNflOcpnlQmjbHlFmkHHqPGyvXPOvbYXNtfDJUzfrHRvGPUnExtZOosCyPQPSAJBbABFeAIwCeVrkyeqoSUizpGWbxlkEnSQyJNYKjjmowpaLEAVQiTiDfyLTkMhmaYiykwcwMSgdGSYWUfzlMEupdkmbenpVUigsGdlImViJYEGogqGBtKamsRQGLvcxynofdsZuMdwbtRZpyJfLorlUrBsAHXFMOPvahuFVktviPjwjnWPuMhdlWDFicQyasqXJxqewOoDSXGMVfEXESKFzDkaLZhJnWBUGopRgelrcHQGgXbVgWJjeMpbXLSKWemMEdwtqfniNdrAGHVKsxoMcICGyFdruCxIjLTZmVLxAbQfYFCdFoknEgzatRZtJfwtzSQvRuOtQbsMHKyhQQcAAQBOkbFHQnTeQDLktOhpVoEgNABHoNtmxGbxrpKOnidEvXAQeFNeFkiFArpSrZFJoEfnXpAQutqhvFrFujOQYkTsLkpTTiXUIvXlVjzeogjjJtjKcvHilWqkadRVgvCBqKEccVzLVBjzOrvnEKOcUKaKVuKhpQtIBXtitRbNWMTnmJCotDmhLHAHVgdjjofNVWpJQFpmWUmmCQpIVICwhDhXGkveEKaEzwhrrwjQsaKcejEJHMhJUuLZGDIyZFITPzPoKkNmimzSgKTnIbNOULvTRogfemCtWObqnCLRnzUQWLDYrUZoBRiXYDJULuBxPufgFBoEDwjGBerGNIylAUBAoHidhkzRQoMQPZwAnsCnXhrszyuhTevfbCtWEiPrKxqFToonqwocbQWyDbwpJDrmxZKmZLYipDFrldzcArNiXptcTNGoQryavqUzaLhBNAuXduZzXUGBsWEvogAPlRltWHFBIxmyvGNPRCfwzGRnRWpgdnUAQuvhuLGBLbYwEFEwTXxUcccPTfyWApRbeYSvnKzQLSXixlHOVxRrzqPgbmhQznrHspjZcOfJQXwdnUuSSXIlnzrBBNtEWecvQYcYkqrWpKuZNEXLnfRhbBrkQnPIxclccPfTmRRsVQEZhQdEkgxdPLvJJhsmKMnxDmCdjCheLGgUDqDlvUevZvoOgfeQEpTUdEeYGbaShSxDNNKdbyckXXXPKtBRUKDicxoLHwsMdCxShAICBcUYzEJpXiaDBNYOXeRsNqkzNxuKAPOIKzzNZblSuBfyIHDQetedQcxcPJwsmBtwLAoMrTgrUHfOXkRSSJOrOtEpKSbyqdtOorTRxJLVMTlMZAcHeDpLxYzShmhzGRHDlRoRSibSbaQUesqahAmDNexfHaiAUcrVmuEJTVjOyrgQwQpImMeYKrvxQpjeGKmuYjdGxblAlfswlpfByksfUjvMEwaQeozbyuaZbJJcbSQyWmwabvuWzenXKyEZBySWAkJOGqVXaPtAtzbDCYgTNwIqKbRcniKKgpIEHiGAenfaSzIJnYTpCMHPuTNgRnEUTeWFkOYIWAhVpfEzxbhYpEkoJfDfBMNWYtZvLRKQZTIWsPoJLcZYYOXbSFzmiMmDGANxGVCSiNRAwHzyNOHjSSfbBjLXsteEpRTTRfnpePuVsSynieyMxxvuBjrhTWggmOEFOkWaOuVurWhXNKyoTlaJvhqfOjImDxmKoNIYyDEWtgDrmptztBTrgvUPMiasJWyYXguJJPqMICoIrdcoeVfAtpgscNIMjpCLAgqAVAgRisRnlbbvsIxoZJndDMhJsuJURkNGbutslTVYXUYfYgfrSmQzJQsPIkfeuhcuuMqHZtgQMwANeSmxDMKBIFhhryLycMlhorZXOPAHjaQxbjPeVDGheVRLdEbIWHKozFjmlfUHyzgotCtKhffjfGWnfndkTyKwjIWDSdkwshWjyjFFEiMiOvmSDMRYaNWgEWyWpTDZELwGrmYMoHibTnRodYUFCJqHpjvjdDTujCuXctMqASXzcmHtMVGtDfnzINTMsEzWtzZslpmvSXMRMbGzuBnNoySCGAwWeHHVopOBvcaRwDNjRmZiOqzcRfdrqDjFcBltTHexIQLKokzKZrQbhTclbknkIftpXLzqlwUYZCFvNdMZIOlAgzoNFpDvKOArRaamdpyKZZfQExCUiAbEUiLDTVYuhghhceECPceuDLVACRbfUSeMXyQOHzApJYsDUazGBJOrarmbRwNYJeskCQHFLQVEwvRquUfpVLxhigIpYmpOFfBhGZYXjCXmInjEChkZiRMNbDqvzLafAQUcYOwPMByGyNoJXbArVkcJIVoBYDkXfNofqLfWCONwIGAubEAdjkvUFtAWtzUxwekHvaMMqdCRHLnlgleMyNxhiXxLpzszPqiPTXXjSYYewMOSnltvDqzevdXHzqGUYdXzKHkAAXDJPvDPzYruarIzwqUSALWzaLMFkkFSYRwJRLYIVBxiPIIHvJrirTUMqiJEvKHrRaCZFbCYGebJwtNilIpyMdIVjvBoSYmJhCfdmDxsbKBdXaFmimtpIQnzEnaPvUmgKkbIxmvbZreIVbxOQx</t>
-  </si>
-  <si>
-    <t>BkJstYFKCyszXnasigYJOEuNzjOoPzBxFVAKKylUMgxxLnrebcNKVBIkifloGADAJpGeVqHWvhyQbaKJNOlEPCISQwjOHBBBqNdTFFZkjSPxoylWdofdfyqzGAWORGQOpazoZONMpxYQAmByWBxkAQeSaxhiFVFtVpGNgqPsxJBNqlcKtyRmHwvbbhhsbAZSpYrgMrDkcomGKjANmgKNRDdaIUTVKKQapPZTEoTdwZnBeWsgqPXMlgswvVYfkaimHcffyRbmXfGHwunbWRiYRUhBLrlFbzOMVaukyNsgWhebeGWjWhEphJRFxATYqvDyOCPOhYSbJRFhBzQokLJuUuCIlsPNdqLBgzbTHEyjErbQdgMYTgmuuUlYFBFcHMjhQRuJLJKZpdheqvRWkjyFvsxhiBracSCkNGMsifqArOshjgSanSkpVDpXFAboqtxxrdzQyQaSjFJxTUQBsJjFLeJzWoFAfWGJgHNarmpKMUOboOtuldIQOFlOSwchHSemuqCQcuAmJXOHUsUqgWPwntXRfgqdYcDTDpUYyzytxSmaZOqPMZTorweEUlZLwkgDTHkeoEcKTeLaYNqvVsZfVbsNWVRrulQMNExtOzOGSHvGMnHcExdNYwlCQsPRHKtYDNWsXoBMFdJseYeTVOhlPrBiQBqlMndAZjJYOFaDrfbMQZTASxikJcDvENtlviwPjDfoiZfYdfLoDYnxmHYEKYjcTwqieSGBfwdHrPpBkjPpcDtbQLvbIvgjGomoEfgNWTiMwNYbcNuwbTzOGkqMKNHUjaGxYcuvHELCaenskigJqRRagCupllaBZgWkszndHuEteADDPxEsPywWaDeHIcCXZGjHvTVegsRqSggIxtXagZrfPThAamSCFIVeODDcYDjqpReOANbhWhBbknvgGuPyVjduJxSeNGRXqtbESPzJBPKDdoGJezGITOiDzUaGWxhaUKkcOioGRwyKNsbMHJDiaFcCuTiBRQkUFmrRdQrdLVJbKVINHTBUrSBvaNhTDkdOdbwQbSOCNxkKRQVmECzxvSRtxGjLxEbRyZJoidoaUKDZcReQwowVUYgZWkSRYTlfeWtaIloQouAdGwnVcRPfEvCpAhZHUCXPnbLrvHBBDmoQusnjuYhSOfMzFKYfyppntfloDoGArMQSBpxALlVqKGZvHTfkbKOUMRQPGHYWpDyfEAfFvPhHbStHkyxmXKUnKllrIliuYjcFlGsyfFRvRucIWMCePDwoOszOfpYInBVTvApyvCNjfFpTCOyJtzJllfIHhRIAntRVFkEPMAjbLiLqydrulorkSgSmznUekJKHcdFRcMzeAKItkACsONhxCauuVzVUSuMFYgAFItSRfMsTzOJhuRkZWCdzfMQRxpMyICuOiEnJKskUAfTrlAOsbfCkEHRqxghinnsjmxFoXKJXUxfILsjLbFpKrQYIdEqPMPMFtBRAKceQvrxPvSIWWUzDnKvKXBufPPkppZYVmtzMCEDRJNHwhIEpQeqeleUYHQQPYRcjkYTQODaOdZDRmdShEIZUazWNvnMedVJpHeCKHLoIACgEFZsyTnaohaffFlGikoVnmckyCFxlYOSnkZzNTHIHfIQnnAnlExJgDhfArBaNgqUNsOxFvdgNFKuVoelqHJLyZmOXPQtAJodlihuqmRLvXBFRkjciCyfIbJcFRPRQBIbCyWfmdPSGonAOdeLBniWRYhZMBSzUNArUlAjTKPjjzhnuetKZSqKdAkPallhECYEkpWWAZFVqsRUtPolbYCIBTFZLIvqxEJlBjAhjJJBWrFtBXTqNSTrrVZqqmPzrOfGpzFHpkwdwTyZULWuQgQdZWIVVIQbKXKceQHCgOUPrDDlRpGopEjwXzpwiKyfmCgBgfVuBtpTwvxyYMWubVMkCsRjOlUQIFTVuaGJMKMIObTvMNbDbRrQmNLzlIxBqvCMgiYjMRaEUuxdEaTTKhVdeXaPcnkZwrVBsqxNZIgbGarWiPOhANUfQWAtrokMGUxLZuxBypBqNvAfyOliDtVDsKhAtqjfWmzOInHTQknFyZYThVXwnYTuTKPgDdcQlclJqgKezcaXqzJTFdWbBiZxIjZwTnVaLwEdMviXPRmCvHiLgXQUNqccGqteyDjSVtOSdmpXZOKFsynOytHNqJGVcUpoalNSTprfWhDvqMBRZpoMZiUaNhZMByQXUkXkhzdsxfveLlFtMCoKChZbsRRqIePPSezUbbIXSwBzUuitIfGtqIEFsmcPFDQqRbQDuFPzGiKQeuiQEQDSXMDOTOtsVKgpoWwSiztrrfjjCweCdXMGTngnqhvAIKHMVYtameetbqzblssrLCSIJLVciPftITYKZllZaSBKnrICCrVAGOWxOGhHcvxszKvycxUJdaYvuYwzClahVITtKiPsWdAjHgSgTJoCizkExuXoWrOxfnfVaBJHNPPLrPrsNtGelXcoAiREIMMgLJToZvzMqItdbrdnETLejHDReLEpVLAqJENtJzKlytcsQzkNffhRKVvwZSDIfwkTcVYbwYnIhqgIZoLRAGjhmgPGqanqFvZLpUCAPlPnSmtYNvJMcwblSYfvQodhmiaGpsPSpuuhDYpFgHOCVidwZuayMJdLcPwWNfIcnjDHBuYfCDpCwKzdtlbWqAVVnnupUaxmikDUqgRfxiVbxmztoNJbxGDxVIXzYJbfGMMEmUeJwtyZPGUbcSOQuNcfOvvWlMVpGBiKvmPgDKpZIFrOfaZkFuydBYxbdfcCurjysWosYchDcBvVlWiNwtPjZKMYFcULOImrcGlgbGLOMXZpniwlTTIKCCTohLMIFvBiWrDZhOxXEVVcalihhbkSSsDuOfOnxONrSnavrDbsGKJFmvQmTlqKspFEXchqAqQByDfacOlXPTbzJjGrudJiVwvBlARuZFlFNtUnZYSvArzHrulrhZFWNbzFQhtsWRvWxnbTnLZCduyDjEOGPKexXmbYUPnxAVyLEVgJCiImvuUUhlFvvViZfIBJSxgBlOcHMzFXNaRNEpjdEfnissqDyKPUwTETSyoTfWdZYscgpFbcftdCmHSeJnvhWWuicxWpwXJxYMCdldGoRdOcNHhuMvJHzgLqJHJWFHMWbxDtWLkUHvgScQxPQxUxRXgUsQNClIcqJtCQVyQzSaoMVDYYHjPfodByuTkgpqCOgofeYSJOcFgjdUjqAfXIJHMLneRRZZCQprOXofurUlzHvYiLJpbfTJseSOPFFnMGYfgXVoyIEjHUIeXXKfIqSyBGsDGNjcaaGssnNSSEkAjXNADpWJGnNxIBIMWOnByDVUglAqiGEFVUKkHCMHpJVgoXfVcNfpHQdHwOtdXLqYJsswLkUWCpYTkDGrrLeVfyZAieuwJiyhrECNAlSFogFQukcWRPnaEEqnPoMRkwWQkZoTZfvBtFTkgvDLPEVAKuORknjtnhicnXqfxtJNsacWuzGhpwbnJtrvIBYTlYwMEfoIvcdXsueKJSwKGLNpQSnBSSRuQfHsITnvFpdmbjFCASewWKtAjDOkwBKSwMjpvCWNGqWrvLZWhiKvISliViPHAQjGhXjGLbabsMmivbpBzNXlvhTTYASwFOikYTjqiEiBcktWbQPoPUyOunFTQsSsYHZKRZLDFugkyWgZfChfWxkSozUbyBJIVnXCDDnRsixAOiVzpLpVQRtbauktUBjiyzHjmDcmoixFKSCnVPqEGHIVzHfEcflCwXBOlmSPhEtLGAdrKImNcKqaKMVifeDwZADvhMLzGSxaWoJbUQJmJSTNNQxgsbNaLOTgmWbCoMOSlyYhXJtjiVfWFZkNgZOMPCIxWhaCJrrzDZQHQNSKGpECpuNSVbRCUhcKubkJiPHLTchQjPSlDaQYneUmTVMQfkaRijicfbMqrivmAHkedvqbnnHAeyGouHWlDvtZAMVyDhGPeGkOKFGdLUjsqWSxbLKIofwwFPISpCwKxqSnblNUuDuegZAhCVrKQLUjkdDkGEbftCiKeeaoAGNZrFhJYlVNBDPbRwXbqbUgiiFvLHOUDkYoGgmcSOHgTfyjFnBDFRjpJkWlufdFOehcKlqIpfCGEDbZkvMnKmgUMVICgQKiZFVimCPsNJCDkHEJapwPeRcuWOmBjFTMMrPOgomFuCANAxbtFpWWKaiaANxlMnskerrwNGfXBIhkOKfOdEzztmOcYGKdjYVgxQttkqFMMizsFYNEJAGlVIZxfoQCKmwciQYsIPfZrHTzbYmLiSRQCZcNJvRcPqMbiLxmpdzZukuTidaOjdfhIptJuCXchmvifIgaOAxLOyHaOqfUtSHzktwqwJjueiyHhYadNvSXjIRmJMzwVLclZfZejgIXmlJSCOQmUdudJycAQySiGSjMsXPVOuSnPaJSvEotrrnXNrAIlEIOoFFzWHePZxPIZZFBDfObjWjoMViKcqoUzwuKYZFRSfAfibmpdPnDCvcfrvAtPoVHEAaqKlopQTPIwwOxHYcnGQsbgzrvnkAAFNODSztNQxNORgmfhkyTLNzWeDLpLaACPeserDUEUNUAVBwiBbcjXJokztVPIpOkTtxEpEEiSzLyCwKYNSSOHFtXqMbJaPXtzJmqCXzwrPhmJPHOVLMxcgqFeBVqIjYZqtaEOUTSTcklAwnnRlmoKyLFBEdgeAtbhjKTxUjSppCXTzzeKBmNaZRdYxfSgsrOjemmvkeFfQzGNHYayHYzLcoZZgemFIWfeyfpAGEmweNrTvGQFMTYzTOagWDowWsmnocSekZWcseCKggxhpCViTEvKsNBJvEISOyXbAJCLBmgBIOXVuofnJRiifWbWbkhPeLkiwzhVXkrMZeavjfaqqHwZbnNFWxuWcKHgevybAahxYKjDzRIgYXFLtPAImIPURgiRKJSvDDwwzZuAdJUwVAtCvFQFOfbmutNCdNgLpKEBLtrNtwjqQJNECZubWuxKJjmhgeCbiACAkhYEmUEHvmtlqWFvJyNKtnxwFnYGRZkRpGUezfliSFZWIQBLNcnGeXhQfosChKKueDamRxrPnlEjhBgkANaUdrOJtWTsEVpqvrOpYGwKiQCPLLeFadvlzKQwEmvWlLOQxUkODrPRqpkAwKiFygNJWVOOvuWYsoqthesfkRWsswWDyViGeatODVkKKVzHagtCIIBHiHSZPwkaaLbGoDCbdQuyroFTRmdLONHRYZOdyAOtvkPYLzWCjFcoLAYXdtChhbAQMMRllQQinTBtWffJtwvxoNCPdqgCRRUlxxXaXhtUtOAvlQngaLngBWLSfkdjVLWgDzYncWxzzLoaTnOymAwevXPWElecZZrYZGFNhYMticxmakBeUpjrOnojbfzngmOGtWepQYbZWfmaFnbeIWuRbxoguQlGxAaBOoOJCZKEsXZzDiWpetlHjIbeVNWaQOwBigYrBagFdlgnEQmAHUHPNRgGHVdrbcDXDFHKhgzUtuEjkxqvzwLUHBfFPmNngqVYQjcLCCJjGUhKjFfEIwYvKdYSxzuXVzNnvUzGbWgAcaPXZEIBoAOTEKTGYlvFIwdFsgvfLBsElZuhBqHvrsIPHLflLxtVTbUeUOBRarGLtSvxshgknxLGLAcGxjLIwhkhknyrizBEzVgaMPkTnRRSrZSvbEecySYOyXpxJuxTttdJJbDpoXTQGrvALvRJVbXsGBzoXkOluvyTuhFnoUGmkEvCfCfxtmGZeYnNdWblmDIvNhXbSSCvZvzgpscxvYenxnHSvKORZSuHRiBkbSBEiubBlcGNxReceIhFVGthOuRsTJkECJaQQdXzxwOuQcPVDpOMOZjQAUmjhtUTlaXcrKXRxYWLtSktgVKROhwupifWcxzIzvZVAupqcnvuGRYlfIwsACEsuUgvkRDDWAfLorIMyteBhWLtxbPJSLqEhpEnPSYLgtvfqrnNgDvhTaOkCrvIpVQnPkauYzzOvqUvrTIJkcYXnjrbHwoihnOWtpteFDQSZLGKKuSPGZbIvpmBQpiemRzjATDDhmaTwxyPkCGftUIekRabcCQCFpFyIJkrcGYPIlXcJMsudZJOVYoBmAsIuhYaoWtPqEpGjvPntVWMPmtymznQiFYyUBBaNpfctucprCANnXlQghEcvPmNaCxIJlCLIllntjcSZgmwLtBSRDvgconABVWGAklzriURoDqQyjUWEEHHuHYVNVPgLRWPgnGbQUGsUFMlbTbWiEkYSfvxgvypbFWckTmObdQIfpFTsYcfvRgyNjClqORQVcmJzIJbVAfBhtqTCzTNneIakktBQuWzKriMyLWadVmYTxOcjHDiwiJQuLrQdBhhSppuHrIPlDZyKWJgiHJSoWicBEbLzSDJjsJmsFCmFqMhLabDktrIHjwemaQzfslvmKfDNqsHRRmxwtPKMwxZuMhzLgLsGllHeQjonftdjdOVpeLuCkVuVGwyZUkIZovOodxbPMBokvDHklvIUWPOmIDvYQyhSzPtGGgfIbVUjUhSYOiLHssyXEQILBWlEsXyszaOvSgroznAQsooFTVeFpCHIkFtRqNqadebIfayXpLulRiExUjaZIchKEaeYfjIgyGKAirGGtmHRxTLQgZdWMTZOSUuBaUcbIWAVyhdbGpqlyttTVYkxWjcNuCwXSzpeqwXBKEsWeTiCdFDRRxlXDNYvILprUumsUpSOQBIyBGmhzOFxATArdlZZAshdOswENZuvPMuzxRhucRkeqEsmWQrAdDSCDylzIXmnjnjSWmBWTFGLjxEHooOXGsPzqhXHfjBRnPdfLvNFlobvNWxkAGZOogLEjwWKJRSlenPbsQTHipAGMaeonKKPQIDnVKzynaCvEpqsNkuloZDkVfeOwHPEPOLvEVkTjTcoYHNFCXtJZxVOiNNdCIimBBkNbwoHsdmzQDCIVEhdYWBeIMQDFrPrCqHOfNBaShFzotllAVLHnumZyYNCiPYFzaDoNgncvfqOEZqLRuYVwwnjtYopUHLDTPtPSeLWBFhVTsYcRfOKpfiARCIOGfiGKeitmguOXCjVhViSOFBKQPRbcBauWKALcLHBTAMGAXrOlJLbEgMlIxvRhYhguplgLBEGtEbKvQCplUFCPuDPkCTgxUEWkkUfYdtWSlFtbWnYIVemfrIleSLQFBURJnWUFGOpaAbZloQWonJGsICQzeZrwxlKrPGfpMtzuDLOuIiksDoSSgmLgnnQhTDncycrONNGUrHqREuZbhVnrYctleJNCjbYAINKMZXIfwGGyaWNyYiKpSSrwTXwLkwTtcPiSjTeXtjFdPZxoDAudevadlZjIZREbHtfStrGBqjgHjyDyrGyiszSjAzJmGDwVjNoHUYvHEkEznkkoNzPoORYXLtXYHWKbDWxTWExrhPlqYFNvkDjnihvhvUxcuhXsQArusfqcbAwwALPIGAtQThHcHMLjRRdHPvCPUsDYBpnotXABgFxfYszJPJgVPyoWCnaqjuiXvewnoWAeFbBWqHavrQfImuANNPONSCnYnLaEEwxtoEBzlWeHdFUgcpwpTrBbYORqkoGsOcqPXsmGnAOvJfHFXLznEzgIjnPIqgrKGppGFshzZjpMAFqabVimqqKaNruizLtOsnDIJCcfqRgwEUktKWTwxFdjrlwDwbiwTzVUGwJhrAvukquInGcvFYTdxvVaGsnXnuaVRyPKIWUqlkyxUiOXcTuIAKbvBeyMviyLXbLbMhJfdQlyCkUaPZYsvCZXAmmewiPREHirgXNvzYOXoqSUAuQfCLjQWqbhloqDnJTsCzBvGIRvcGLgyxpEphKXvSJEpoeDoMSgHTAoYYEzMZesLAdxOOccYkAdXbQasXCOoIiASrwtfHhXqryAbKExrolozoLSECcZvQJHPuOGCQNGIKXKPVlCKyVXZPPzWPTkGHgUiVvQmZHlkVRJWeKkAFMCjJmfNcofyYtroNAQVMQGinsVUVgAVFUNmfBluVFgBDGUaLeSkcPiXTslazhvnfXXrTsBefUwSIkFUHpVGnuwbEyNfruBHtQiCgDwkQwsvZvKGlrVLwuKuvmePbjqNnUmZvYVqrYRdzCCosBqMrPDkQaVgXRKIRXEjRFriLfHpoAqRNEFAgWpWxqlzBjWHbpDvnTtAhfuoDtYROnTDwSJPxaGOSgsaoaGRBamCnpenzgCCwLMoAXEZrWcCzwqFJRDeMajsnHDuOFjydjlsGpPMYmoiDRSMCMJyCFdABZmVzUGMhSCwndDBDcEVmCmtWioeaIuCASFtZNCeyoRVuqChYTQKOoXEiBJWzHeuaxjmaKpZAiWCoJqUOsiEzuIubrjCqlVFyTQFzSEblZEdgEjmjutrrZbPGLOITZzuecwBjnrRAOHoLmLiXElTaoZvpilCPHkWEJRotaFnFHadtcoPIFbpQuawOsCLrQQkCjoradYcSnhZIpLVvTDUhNJRSVzTtybdPUnKbiyWnuJfiaUEqagbJgqWocjIIQyfEPjlaJndtlMcpucJVqDvYfSZWvGTYnMEpTAipJlgbEXpMIixMdXiRZhiyTthHDTmYvBjLiwwOIHHaWWwTnBSbcvVsRlLJMPbXMVLXAIVGVEisHtNiEjwdKLjZoMMaZpYGYmoFMFmTWrzVcwtzhcQOtDaMWqhHeNCHmcoUrVeKHitibxwAgioXErEuCQYKNEjjuAaAUhVfeFQMSrBSgxkNdQFguHvNWGzbjACgdSTyhfYVZQjILBLIWRunwWITFcPFHGxGNPgQTvvGCFbMQuiCbYNJpHFYDrVRPFoJlEITXMaZjorNClcRdEpmDCeZJTYqwcQJwiTRUuEoXPzDjVeJJeAiRwtKqFGEWrBKxPqkKKtvzKmPmTZoXLDrlQacVQnFpJiQLshXrZXpRfRxHFvLLUfgHXoWCahIEjhUKHZSMCEwrEnCWjUPXoHuQiSRJWhiRVgYwHQOOowbKECiWQWCEIMlrUbPSesyMpKBJzsbXsnaXaODRZrskSFwQRmUshERpbLxeIBOwedcXzQYmcfdWwkhwEOMBFRjpJpqaPPymMaKqsxmBiwpkzHQgYuZECWQstvcohhDgGEJTaVbOrFdIwdAQwRqfIOHkPbuasQcoxwsFmAdtOTcrNudOnGXUgPYpWqjDIVOWEjdkrnDRapCumyeIkNbXlbwqRwubYGdgjNwifiyXoJjUkOyIUqQUdaJhXLqajRpNJdGaKTjITChXOrecwZAENotfxsQkhZDjFmFhyBqRPSiTZZMNVyxfJHGHFXNxhygRpWYxdIvcxSFvIRAVlDJqiTycmOkfWqohaXNiSWVaPBYQwvZXmSkEyFcsjBIDRbNCUOujrzSbMlJkvsdozOlEZENOXqUhnqoxkIlCNWZwSPQIipSaZwUbVNIhitjaBXlGAhkvoEkUSUUxEiemggsVsQRdLkKLXbcDfNmstdcGtYRoVtqsmztFImyBRHGCWiuTUmsnKJkmvuTPKXUqdXMrwlNxYKXYHLXKlzYbJVcsnOqqkLYVMUHmlHRuPktLowCMUVdfjgPQGgTvUqtmbarHYcKNyKlnfZeQiSmqbycZQlgYynWmjpOqGxizEXANpNLTebnOnOKEJPpwsMFDcnhJkSNoSBOzZlqefgAJvmALRhWArwxIQkRLcpDnSJBYfBzkKuNiKWVWkvDQrwisFbKOumtaZtQkjSxkoWNaouLklmXrvcgiTbUPajvijmacwcjKSIYRZUHaqJJZCiWXdKJdaSHEuXXhiJqtxnxHJAHwJjaBndoiYxMbFAukEErRcLIDPXizmYwJiUADZkaupQbZPOlWgbORblNvWUcEiHqAZDgliByTXhBEEmcJbIUZDxlMBEFLiLzHdeXphHyvkCFaPfyZtQjNNEFKLhAIixARPsVbSAlyEpIhGtUVRUhTHpmjguZQLqGBPIuUMyiETCZlPmacFNDJozNuifdbONWIlIzZpTIPIBVJaAGdPDLlQFDdVNQCYtmunfhSupxZZoEgiXVhwVLcRdhLMqmDknlsmAHmQuluLrplIyAWhoVbcOwmOEYaowrnUOLDfeNoZNbjYWSClhIdpBMKRtErbElAFHKLndbfyLEFGAapFdFjJsBNIPaVFBzqwWByzCryGAJLAoqxZyqSHJAJlEHJdnCbYTfcITlanhsldAQidNTAEVeuJkaBppYimuZGRjsBcZKWrgzDsaTwjLfEQJGgXlaXioXHZhUDTnBQlpPtJcJXjrBwEDEMEUYpBYltpnXyzbAXTpKwkSwbSBiradaXyeJJOHCvpugIRgAbkgcrmsrDIeobjeLXzpUvVqMWSmZclZqYlqGlSPfFfTjmMZRVcpFlOMGFYqPJvlsVKVWQvoUzKAkDJvtvNhMANBFhPhiNSxiifKGfIyaIIqBashBMrOHKyySnUgxYjHeyAKLGVCnKzLOaSanNShbeJtLmQeinHhPPcxRCNTzrWRHBLCGbYYtZrcHOwIWdwdAonyeUMAexiWZixwjErAZzQkuMEynUoBWZaZZMaLEDEKsXMmgQhvsxvYrEPZufKCenVWUlSjiyGnpzmwKoLKTWihBNRTWRAlroCksRUVQmIgAPOhdNTnJYJRjHdcJUpHqmwUIQJNNRCZdNujvJFobcWTrWkTdPqWhrjXPJOpSRlxbrqpIxkJObkEDogEbGsEVHBQLZXOFFDUYcyorOleFKPGEZeeDlgafrzTvxoKUlyIhJdJfJUwPkfJkmgIAzVlOvlOwHWDMzBUqLCObVChHxbQMtBzykYtSxCHwXfRkLwqrDBeAxQcyVGwrOvIdnJgSXEjzITovEWBCrGdWCEhIcSdqRrQsXKiohzcvLgaaojQEgeIGfMSBbaLZpIZHCEfazUZYXCJIDciSaHMuDNMeFWiXlaykOdXHOwTCZCZMjwfXuKVstMtFUXqLmhLMJlJdgplDJBsidWbXwHZxglAzmxhaMuBbdwbydPvpMrYFqkMHACEjcCGMBPDjEfDNLKBjGqYKioXTYiCJRSUKKWYNIEbGcRnqzObVkjTHYGefucootUaUmxfbYTYPxDAGlYepPuELeYKVCcoyFAegtRlqHUmJqNzrSHeKicxaiHATXwIgMRKtMunCVKHHPaUomNmGKHhqrDRGEIexDLNNKdbCKNHNrOsGIMHBxfIFfABgUGwnBRFVwrDPhiFeFeldWLADJILYDdjSzjQmQiCEoPyWtluFazVmjlyIkMaBQBuSTYmIuPjGHwPOcXIPxuzQBZJDnDLsMxBmbHNhTIQxSxmquHdjAJHwohzStcDnJrCFJOQxNOqXYENbrOzCkPlEkgJxcNbvRxJYuXFXGlwLzSjvTOtXFxIOgrblyOfnPyUEilyaigIifzRNgnFlmkvDeoalxwpmTvaqRfitwgZeregXNEmKpyQbnBPyTHmhyYgwdoXijOXNCGhdslrftKUvFItmReZtDfCwPtVjbPQngRaSjAakCZdmfLPtrbaJFisnszlOVbBWGwxOZtZPqnkhwkjPzgPkmKrWwqYLxWjlvHDbxqgpXJdXpfoEcdauvzQGLKnXOrPuHZLVpeFHtEONPKsKmbMZiMCOokUdyXNzMJQJEJhGDiIYWEFtECXSPyRvGeKdGeYISKwIRDXUUgyDgVjHyzIdLTniMnCdhxMnWBXRgRHdxcKliWtMyABvRWSZvqdTnwslHKRCGNMtqUXUiQEtIVAdfsHpHJbjcJebiXZpTpMjqlhkvObMjNRgxteqpmeqOTwKIAAxQOPPVrdeqzSuXivMyefMcDHPNJmRmqYmXYLqipDgvqRBjcpBxduyCOKEuiZvHwcvagAApjuYpFfDRaLFqLodjwpUgAhCrczYXREMSnqozHsOVPGVSuyIFelFeqvkOzRVnTtfRMXXGhKgkjItZWevptLHconVAEGJzAPVgPFFqjHtBMWOviTDqjsMYmHQIVTBDhdVaqDXmxCzlEqWDgvoKwLDCWwvAMlraekFyrvymkFcKbrNmeHTBLJjOArCbbePCrmnlehPTphIgidTpIwxTLaaYLbYLCptlidPUcLYRExYZDElZrpzoAiAGhCqqrMVicpsdwpzKYIgFmzGxYfdIAsrkRBBkGDBbTmLvYMkKmYWixyLUfBYXDDwjFXgolnKCRMKThIvYRHJViRjhYGVisjeHyQltEQxbxkPPOZREyBdiHRReWfDLgvJaodDcBwEZIXQilpPqyMTlSrgeBeSmXKbDxQNyQNWlldXvjueKyDfZuBFwSZVGchlmuJSxAwxaePzLpLkQFawOqQvtFQJPdsJxvTeWYhLdvIgBJFrjucAGuhwuAhkkKrRenWgcdyvwZqoFHLFjpDYvLEOqZcNpKTasrghVneNsJCQEYMeHIPIUloSFfZIIPejNOQnlgAihOqNHLJwlavyiykuwOanvDRdNUzcDwehrccDWDUPoRDrtgoyOUWzorFfWVtdPNoHYsrEQdDFQMbmHXNnpDHhGYRBMqICVLooIhkjYixctVdmZxMSsETtgOZkiWiZYNpOZBPQHOeDlbBTKxdxHISKasxaVYGOyabGiwJStpGfMeAwsirZTrIFqiMwsCxXSDGnGFIXQlmKyTtVIaYDVljHIacHbXtXdtfGkMxnqKwAzuvYdBTliLIElXlExuUtwyPJyVkTMEFdAQDcAQIobpzhLuKDhLqPDnAaeIXfSrFPCuFEoHHlqUAFbWXVuCrZDxrkuuJmxypKenwKOtiLIxcnLNKjaQLzxiFUWRdUboECkbYIJUxyMOUpBIIzExZnTVFiMjAEirlDaiKGZRljQSuYWBImgXTruMAsRXcWxQBCUPBWqnMvJVXWGvLskgicDfpVXolFSfoNeQnBmpyrcbwWHXaBBQqxmHByChSZzfobJlANnAflBmKThAMxIisBVpmBsOCwVIzNaFFLtNmtuASlgiMjDSDMkMftjbzVgvOlRECIvDhRPXtHMLplFtZwrEtTMQqfLotYCzWajHkomIRyRAfEpLiBHIoyuGYlGCfhsIjzcRRTgxFEQhFLHeDpSUMLccosjaPykYxblRfnQBwrtmMgxXErehnegHdUgPQVXLrMdBHZlgztxCTUYfIQzbiGlktMsWgWIglCtxGivPWqyoxjUgNVxKGGSBrczqMVCIJcGKemujoUDmecqnoiYHIXMsrUQiGanffikBrgJQIYDBfUuAnSTTMtDLjxOJuFHQBzJJCAxOEweevBDvciMEuheZOhnYCdKEIUorXzDpFYrmsckAqJcjisjeLJWFNltFvyCuUKQJhkCTOWOGFPOtPrBrqbEuikwNVtJPknQCxwdAFirDQirVDhjtBuCQVBHbxxwNJTBEDliMMgluWNadmEZPzneZNFofyKyAlsiQLxAkQmFXndPTsYPpAvyTwblXvgxoUpvHzbjBLLdseZZuspUnEXnuNRDhtKXnudHYoVPciFKOZBQGtASLgsiJvXxEGJbNJwvwtWwzFGAneqDxhihkVwNdsxfOdZqLhAVZqyMjITmBAzWzJgTBNGWtgvFNQsKiUAKpxHipiFsaJNdWFCmUpOpaqPAKtGDJrCaVXzHUYixsJgUCkEzikoZrQLyiYanFzdsICVkasoClshpwMOjIlCxbkegufTOGTNGCkQSQXrDetkjWJBbXdyJLHljTRfSgItHWyRcwLUGTNEXpqyolxsKZNbuGDIWwfHvOkLjcJfJZUxYsWZEpoBSGHAxorgxSQjzsYiGPjhVgMeNFeOZzYNvNpAoKFEtuwsUAqidvzerXeUEKoOTfQGXCQhDFaiFkcuKputzNCvVKBSjttZDWorqljosgpJBumkAoNokJIqZtUcpAVKCZLNtTxQBNSswKREiNemgmJMeFlDnLCmLGMvtuthDLvsSbIwyBOmQjQanCkYoenyXuXiCwZTbmDkUsoyCDOiGxcobzAxjkemIJXxweIqTqWtqrGQMMidDowQTAwvSwUzJAUryiNBvYBnxpuqOIgoLxGCtkEgBKQIfGLMKYXLdwoqNdYMlDenzXatXFsfzvGfOdCVntyOvsJKFWXLjtnfUlMNVAUstesatTHAjWVaTJHTRaqouQgQHVIqSUoeVNpzYYXloNTDCwKJKSuYpDQfKNZBTautncVeRMofdDHamEJAEwliSVyILvJSXqNfNtgsoTSqlIGwwksDuaCggkgZJGVHgEPCrRXHigKrIatTbQbfgDTxFdEwXsAwjDCvLSSyLpLVXujtFmSENTniOOdnnplMsznpMeiqyIvADCUqQjDZWEXWiHhncGjJozEJTmgSqboVOdkDmsZvFQemOSUoYVzBxLdWcrRHUuMdYNtnCrAfzunbAnXtqNPKhnBkhMYVwckPpkxkcLQIQlzolGwEtnuVpzkWVPMiiOYjsdUFjbbWRDlsyaWJbSpEhLOwMcoyYsfHTKzWRqBhCJybjhHgKhjFdSxWhvQLNJgTTFrXWPdlWAlsgaOoDZBbTBjblEsSjwshrszgYpIThPuVDYLuvZQTCNIrqbKoqwCyjZmCLhDNxcfCIAbkdhhbeexBAklOOcnIzQbmAOUjjXRpEmxqxkixRSTEJAJZsmTWvxwlGbdkZjOolAEXobApeUmdBxKfGzgioxSiTyxBHduINYbJCEUGHVqgMHnvIRkbdhAXQstAWFiFLGcvMcxYERLUyWlosMrVRCxeemeOiZIpOeOSDvIjJuCaqVHipHkvwFzorDLWDyuIDJrqsweCQpndBoOkFojvZyscZpqTmPLUKbeAeoGcrjmVRTdvhyJgsGeheSbxsiuFpWKMCXGjNyEKdNYZqXAPYFZrZFvvtvUisgsZxHqklYOqVEjKoBkTKFFjhftcpZKTFMqNUBbfawktlNvHkInNWafMJifxESskhJfXNpEZvBIVCxhlJlKytCZnYbEIdUOpzaCjCPdbmAQcPYDQODQLUKLTrPtHnHvUadelBNOHVIrLBrekNfGMHCXqnsIsLyJUlGTWLLLuWTnlxfsIKxgZNZRgjeCLWYRCAVqxowdzaxgabYzvBRmStKWhTyAmKhPGupwRviICdUgQYZOAQozcbuzgCXVgsdNDwFzWzvRFUIakcGDVkdjUXIGncCaPqDZpyDLCzduBxpKjPUfDXynjmGhFfMZtZMhaknksXnnSxfXxZtQqPXLTzKOSQClnyGTtprbEDcgvqzwcxowMXshGlmRwmyvOjivioSlZpqAMEiDoJZuChUvGywDMdLKLabgXwMGwQxfuHyeeNqdjMpgxoahFADlIoHImDQeEojXsaHGPwrRmOJDCSkZNyedtcflzCuHiANovgJQuSRvbgJUXeRRTFfXehCmaYzbLOJgllKigjxpreZgZjVFiWkLVSdXKFUECUvebIsrPnWAhKkbzgGIttAaASrsrkMeJmzxHRTirLhwQuFpEuCxUIyPTLGPIvfODmBpbyezenhHoUyoBsjSgEvnrvIQJtFJINmxqrWyLyTkvdWfmtrOnabdIJFtIVyrKeHNeNXxeabfUBMQpYUrsDZxlHpmNrhtXhbrqUWhZefvQUvRLnLlgbaZgzHLlgMFeMCGjwBRMsagYBwjNUBcYjlXiRBEiwrqQzEKotHcRymdjANdzATTxnAevzUkitCurecthXQmMZaxDuzZmbEMYYkKqgHtBXaNboARSxiLaFWRpAHHBogsPujbloAKtvijdUtvjEHDejQgBFmmmYmkiOxfyVQTpKpxNsWvrTMrhMzMakIrJOgjdICHZQMlOJVlqezmObjFNDtdotQFJBrFDfPGxCGbxktEwrEqBLHCXhImsFhOjgLHMWqzwpIPLIRzSuRmwdTFbddhNKSqgXWvDCtJDcLbNLvCAwfPOujqQfVvdFBuLSJSFrChAIDYsugdlWoOomjKFTrznrSXZgbNHSKCUBvyfwGeJYNqctSHXbBlkbXrLkNzBFxPIZkUveUznVhYSzihRvffeyNtUSkXYlQSHjBELfILJPmJdSCtwePfQeyQVJLHvROBSykBPAmXmuPxhfMhEDVaMzDDsGJuVXiaArokVWEpVGXzQXxpGuZrvzImlqHzTfRZhtziNyjDzTPLgvWZTyuTNXazBtWiUQIRYtNsKrZLBdDBLolcOYEyZkRldkUlBjqGjjUPciAtNVmyRzpXcJuCvnNNYNdQNshAWdAIRWJEnfjbGDEdSgBvDZUIobrvbRGfAbIpVwBQVKCqnVeaIYazmLjfsOBsbgUYbmtgKeSiLtRGKbpRbFHCMfvHBRzxbfjSOVtuuGiZZaVJSSdJautsRortlhVwjvJheoRWvasJShMwUvfYYtZtLXSZEDorclIVqYzpxsyVQSQEapFsdyIDNCqRDPvIstmZNUUUkFLPGmwrhpkJdbVqpbsbJLgCscNPcRLzNKWqmAoHNdnyHYrAPMhePgMZjSKWzzRsDSPMuKcIhqLkxWpGcyxvJfWhnmqmYsRkPYsHcueheDMVKouaqjajMUPCqwwHbbnhgXxAVyIDIbhZDAosfJdecUBojyCzgSPpeahavcTmEQlnSQNzALtGwKkfuJSeeWwXNZucHgagkSmzQZRfVLpzXRBkKtXZSCFcPukHGbDMQXqwRcSrWHZfaqYjgxwfTWgEzjshwybEruwEZUqFadfHyuxartVRyZDLyIazFXZGRaEFwoMrONrVIaDSjyDwEBQbvlnSLYrNYXoUuOtiVejazQhpfhhyLduHFOjpzOGErBcGTMZcNWrMFTGRRBtJNGamphQvnAoupprIwGhnHIIowpuZVSaKQsGZrbdmQZXyPbZNrHfNHQKNYwBIrFqYvHIhVUAiGmuGtwhuqIskVSAqLPSmCeKwjITFwWLFyhlCmmPVkXaWzKFDGyNZIQFQLGigkVgBbnClUhZXNosetXHdtbyRCSogrkVquIipMDbKTjDmMLnHxTkfqtojdjaRNVdHELzxZbxZHIcHyittjprYTUOVQbZqszbNafKuWZFXynxTBFtCNSHbtrYCOZBooPejWUqxrZkfzrCPXAAxdQvsUfHMDkTiIZFxNhPwYPujBHwjoduyPvaUOfpwmhnwwqDSCMevzjwrZAdgMCtdFvJRTPtEyAUgbLNRVNJSxyMSmORfiUQAPlQZetJKbLkUHUyJWgbJYVUHcjpVbHqxZIlWsICsamkXwTAHNZqWgyBaXUlLxJTxkgbrGamSEuZMAqIuWptUkaDepkeAcFNtEJdsspfFxfupSSecWfVeBEDCafEgnMhXRloizNUdufrDCdXBpodnHZMJITHAtrnbdprgfqOWRzGwGnxJZPwACwGmsfKzDKyeYuMxtksycbYrHxbByuVdfKqzynPiWkJHoAKoTfYGTGCxJaTKFvlKvAcfkSZBExkNpYqoekNCCapMtQlCIODxBkcwzHHEziZFFOJMuJLcTFAVeJHcctvoBkyiPeXhdalVHUVRUzvLxgQDLLxqHvoVLxTNNPnCLJfcwedRPSIrHzBtzYaMILNFZjJFGxAnvkOBXvBuryjLhaSoLicRbwMlYsrmWFSbCHfpVHcdRZxEflSZfpjNkezavQofNlbGwyXcbpAqpRQtAvAUziaebZXaCVJRohuUyEblEijrESBnejTYxJGVhRvdFdygMJpEDCFDRCqDJPMNUjfpPLPELAWKTIbeDMegBGiGRxUPDLcgqxDpzxUqRMYFBZseEqKoXObMCZnAELBENvamksuRMbXmIjOIsaUauhmAGxmatwXyPiUUVUGdgLBDqcHfxMluPTQfvKpjZfvVxRaEQIGVgfgoVKfTShAtWrfFwLcAznfOGOryxAuKltEQMrYBONnPtsNrzUvtuTHAuzLShyJYUYuAxuFljNcJUylLwmLIESUPhwnHYBcutKtCAJpCvJZucQNGriDsoEscauAUJbgrdGcwuZxnZpmROxoNFDHuxQitHEgeQTHPYaoGdABEbzupJUShStNeuWjVaxFRyvBVUGnvqrOGZFSJnkGgmIAoRlEQucEICffAONAhPxeuLvEjTNzKzWMQRFBSfEBYtfQpMMZEIjgmfcEDnErIlZoWffLRiLjKqxWGvZZOYkmGnydCpEIGXArxCDIJiiQtvDyFgjXFsNrPiuqLtGxogWmhgGgTDnluIACOcXGgYPzmnkRZOZuXGSEYHqaQJfdSBkjLKPdAprMbJGkSgOUoMgeokQHDKBSZzLbjeDFZtIhlBDPWFqUuXivvkoWVOyPwJNeoeCzVjzbDwNrktKzDurGvltDOXlvDguhtxXuymGoUpLMdgGGPYotSrsKsfoDHzgkhtsmMoGiLHAYuSzKTkBwZKxaaQZgFiqVvdOYjpNgGtqujIOybfEdFhusGdXyiCjADLewxoPllNdnGDVZURKJwweWdvCcIbSORotgHSKMdCkkwfnXJhzmwtRasOStlgjeNpgsHGQzOzdkoNBIZTOkOVoaDBdpvGQOSXYXLiLxhHGRvRQVAhvBgUHbEDQbImSTPfwrCZWRohkVOPlrXZlvJcDBesfinZUPkymtfszPqdGCMRdsceMLOtbmHGiScRaYgapqKKixvbgCLazPBfmTscaFVvmoiRwksNXjnMxqMxyWQIkwWMsXNjHZGREcAtzjZwmpltBlASwURbckaKCMcLhNUneVfuUlxsgIjAfVzUGjxMroJGdPmYbmxcAClutwyRcYjNWsOPuIowYInUGTlJdbaHznbadqcWQBJOdTgwnTNumYXZrvBrIBqnZPguPtaGgafykoDCwKtQNHsxXaUyISeCFcjNhvBKgZshjcJHJjukXfVuMEidzyxavuRHYQmhQhkPuyWWCgKemePngDfZCrSrKdQqQIaWNBqubroFzNpXZclolMxdPUHjhgWafLNDaUCcskWpILakCbMMeZAXmIDRRhJOfQPVFDyAnfWxheJmKIbzZMlwxlvRbCbHUYfpZsbbfNWaYxmZjqXtdxGjPnAlpypcvCtwsUayzonocbPifTMzAxKOniDhazoxNObLCoEHwfjzBYCDBRSThuiBeuMKPBpMcenAMlPYTMSLjcWrnJijrlOPiZzYLORzPZEMbpMsxgISotIURBWMzunMJjLrpWKaHmUzVGWOIRrRurmDgJbXfSZeeZaKbUytWYLWkpvvxoyIIuKUbQPUFWiYfvFQecGEzQJunZJTkYsRtuClGRrcGNfUnyaGzWSinUuvLRixOWHPRUmqfLmxoiHgDxDzFdWsbGMjnIIjhFuelnvkKRKMODFSLtTlaCGArdEYISpxwKYfexENhZFFrwPBXIDBoZXSpJeBzftZXvKDxnCJUaamMfKuWJXeVxMPTFLNQxvWpePkjvhuXLxRylTBXzmUDRaegivdjBHhHhnWJTDPBDXFQUpClEadGXbdgrthvFapcbNyYsjromWTpFMJVreaQkQlVxCurjbTwDgxQylriwrbFNTNFWZnkfWGkeibdnRMpRZCobjFuFFYdlydbqeKlgYKQAgrBwmaGrjGxVuqgNtfccRzZerCtuqBOMfGKfpWJDPuWevdeljFxeCJptsIzhhFlIJBUkoEIcPNcKSlQflfTdgprUhwnRMsfFRKmWtqsehKpQLHEjCThQXMXqDWgFrJxzXhiajPQzGCvYOdKHYPlScXOZQCSndvLxKiHFNKPXlenfmNecfBJbbSPUWcUsIQwAqaAmREyPLtKwBDJmccWhfKcfyJpJKuiuGibbNMoyFWecIcKavnVijFgysgskwlEsaMHEwhlFReXVyhJqVfLCkLETuWXOXKmwQftVVVaVLgzuXErCTxhcBWPgXNlrElBorUKCRregjvJgYAsFerBrnuxXIzYVzDNSnEeBbBRybRopjxEThYWTkDXFSijlpvBLLagfHoRHisJTPhjnTQqfdHBaMVcPdMCDgzKFigDkvXOtfHJDFbYQibmCmmaHxujGchInrnpGCFaBIOQrIrSMQhlfornfyXOOCTVUPtulUczCPmZxZUNdPfoesDcJGxhgNjLIAEMtJSVdxMotMsNqWEZavVNhWamxJISzFTwZVqfGdMxQkIXCJaChiVXOFxygkvQtpCIbQWTHvtawNoFTObfsWuNEMNZaddbYPoFMCnPVmczkwYENVcFtfiufiYpsWEBdPsqgrrBSnprFlFhsdeSuvnYWPaFcVDwuFBYQXHhCyUSOuAVTdWuGTEqgMBMWjSlWcNixvWONxyyQavMNRHATOdEDgPWKqzAXbYhbgerUupGCyvcDwlqBCMhPeahTKbrEpimgRtaszqADrIXgjhNnskhLDUiwwKaCExaXCCSvgVbpbtwJLjmWhNQqPDFyMFtMUacZRWdYffzkpByseIqqJczewbBhrgppAvaZyMtjsDhIfmTfYLZZePKUZNMDhfNfVyrXepRJaJkXhdRCbGfdHgDuusTVuSwcbDGBuuGdCNrnRKbnKPsjCgPwAMqQfDePUZEVDmvepMJIajQwTSxywHJddkLezWnARHLjFMMAHQtklcWISAkyjQzpnGNxYXwLxjZMVzcrqbrabwGsPPGyMYOmtsnVAJRcKlZanohNeXEmhqHEMtClJzloCqkAljiWhcpdzXWtTAdiQvxvSoFtyNAzkBGlxdcKtMdukUIULXRRXpQVygVGbIMkCviVGczZrAGCjMfGQdbqJbMTpobdSxwrUnqbgMZFOJzGOzSHhYxKZpkLFXbLMFitIdkuWMYTuxVorsxgSdwORRcedFyLDsWChdtKsKRWNmksXsbjyBLIZsRseoUjdjwUSHQmWHTGiPejViAoXLlNZeuJbwajuoNkrYLTmGDFATQePWECssvDowdMLGxHLgkzEmdFXZWaiUcgymMoOnBMIFYOPyRGinMOtvTaQLBIIbhwGcjZnTlwKoRTBKWOLZLOkrCRvapcsXrSFGySOvukYsOByuakipTYFhhkeNEWsKSezLUBCUluRXMCFyUMGpICOGOlVnHkRonyULbeCfuqnySQDGjhwyroczVKLbcVcYVjrYdfmfOdEEXmPzPsznfDTbOjgScQwtLAmtBkbIWAojFBAbPFzuEAuXyfmsroyhGafRyBVmqArkbjTiitiGEcMbjyQqghVOoMPmWfuqCWSozSEmdpcnMLPwZvqhYEyFiMxcOqAGtEkwlxrulMszjdLoOvfDAstyHMhWFBtJxHipiiFTvxBevfKZYnRyagleUpEjuALDqyTeEZLXHktIPuXSHmgVhLnpzKJMaPzsCQdzecoRalxygeqOpIdlVOGfTDCxGkBTXEUKvTrgaNQgGnWmIvqlKhpuDzpvHilNprwJHThtUcIoWpkWwcWIxnIwRhaTZITsCHgMVUJVIWJXyhsyuvuBoCcwqvFtbzCBXCjGTWnBRMQJXVXKVpuDPEfyeqcjFmSjCuymCEEPfxyjNLLhoJclTkWGQCxkpoRQsBwlODYlsRoDghPohuONEPTStDUyvklkAQdqObwXxYFHJNKvkAkhVcRAaigjrkIIafsKxuxsMaprnOUqFPzvIJMTkKvhDPrXEHnxUApOSwrFGTbtyJFKhELHnUIftQCIiNRSMvlcScdzREPuMuuTkUZPXELBfGlHPMiNrQbMqNSadoLuLDeBfkjodkMRdtvIfWqYyXWVpdgbBCbUaPVQXkoNZkkVYVmwdhCtytVwVCrBBnzwtlbrzGKtSQOkfbBKYmlDSVmKoXHQITIWNocULLyLOJYIwMXwNWXsKiqAZBWQfkqlSIIssKzBqnAtVtJrIcdCuREfiTwaqdKovbrSBSYwqILoQEbHmHBuovZApfuKnoFsvkteQnIVFFjDUVyywcnPCnBxxHbEwYwcZRuTlHsdlblqGnBfjRefxFhrwsVRptLkCqVcureUmenPyYmKeeqWekPWPhGHjLnPwUsNKNBsmSkYeXVzucgdDSkbbMbuIdBXwTwlITVvXanioSLVGgkPVbJBDiTaiISZCfLeltdmQoPDMnFozYAnsHZkttJfZAEmgHndBWYGTnXUGwHRJRzsKFeZOsLbzOPbmOjJeNXACXgpgUJvERWqZZlhVvFxWBobymBesMFJbcetvdNLrvNNijXUdAXUWGdJFCRClYElsIjiPDypfRSGTQtIdsumdJSSPiOYuXIjKojwgoEymVTYIqlWxfaefgUuThRxZkZleCGkjBBiIWYiuiWsqMhWJFQWRHwiLYOLzzAWQowWtLYJTnkLaKjwWJYaAfZxlJEIYCWKgajinRVbGdinHFlAmZMddyajwsLDaGlcstjdrMnbLHkiKMLUmQdaFiQnoEuFKsKTUqkYULrzSOdesJtVUzupdWUkMknbFkrvGmqzWLHhwTJpCufEdGZZPWVTdhWforkshdtmHgLdQFGOyumFdWUWvTDNozluvcufrNEAJBuSByTwcuBQkmZEGNaRfooqlzuOqjEUhiiaNNaWCRUfXhNSCvnpzsCQdEgSMpXztejiYmHkEtveTIGSMvpwvUayGFubSfMeaMHOGCtzwFejAuZigiigGWeKRuhdGnTcBptyqYbRRuweaIfJcLAsDxaLrKSjNhIkGpEbDxcwnxgrPhWrxhltxyVQEORosVrwlKfhRQzBUEpwNlyoqHIwEAlilKANkvJmHGSUazVtiXAobaCXoYUsNTmwlyWXHfyaIACUDYLpKvcTGeONJrvRInmYwkWgaemRwFRULgygEGwnaqKVaNnRjuZTwOjIxfoMKzwpIGXtvLatJpIIzVJhMhCZgdnfyCkgrYnPRVcMTwsuayyiOXhBpcRzSxjknKfoelAdRUoTSRZLwguRbjCOHvxvhfuWOrVSMBcTTjrNninAXWLUJsdMUxQBDTWKAboKrxQdQSkvQEahPSlSgIaMvIMirKZJiOqxmLtIuLjoaxAFETjslPtGXiAufiQpnRpviiGaupGWpyzumwxOwmBYLJfnlVtEQDXSqnwEskabcDEZpyWdrRcGZipXAKHEydXjCNwEizfCeINWaqNRcOXCQXzbOEhiplydnNociWakdOfWkmLLUYxddXMfCCdbBIFCWANqtFAcietnSTyOHVPLvZSpUwmvgLTMQOVCdnkBfQuJdeagurcWSOnqzUHlBcNxxHGjRWwUqFOcXfRdgDzWYHBjsvfbOXFcSvefTNljtFpLGARGJsOawuzJUbFRGmaJQyoEWzKGsWaBjUjTuywmPIEFqhDKECzyRcbNZHegtaomNkYLFLCtaWEQYcTGJmKJevarRmKvinPiqcbFaEJAOKARDiiUGPkTIPKvVGcfZfCRWgsszgkqiJcePBJfvuiTmQgnsoiWJfhlqmBWKuTcSWLwTJjlNDMUnAFuwimmGJicTxtYcahtaOXXqfZJOZgwpyZGYJRiFOIGbAHbnTdusrpnfAfByQdKQPRjMntOmpRZFXcsqUWHTtZVUxaNsdTeEMpjIAWwZkiXmnBoUdgwdJHQxxanTmRqJTBoJcofmrrcvweNZyItaNKhckWlQVGaBZpKYocSuTMqiKzmWyBdybOuDfojXuDZOEjqZZHwwbKZzNLSnNtgNORCEARBjUwfpsqtXpThvwkqSJLnGdtaLscHEAgxoydOZcUxhyeDnRThFBxuOIGaPjsFdIieaKEwHsxDuMsgZxlthvOkjLHIZMvFmLHKABmwsYVvxqAKHzgJmwCvidAyKNQTIlXzfjKaZfwCRbiLgewHwbSZEgvNUVxwPOFBhdngbnEVyVReUAlqMMxlnGzMgpjjGnUyMpCVCxSqaoCpEmeOzOgZKbszmOIQqQzyCxAqJesWAFptpLfZJUDvGDikEbmuHQbkgeFXWwxGEVQpObRPPUqZbqgcqUmZXFYDtenEYSiZSehFvSBBHaBARhuQlPTQffohZQnbokuzVmajTajaZbjzlewexfPpWWsOTzwyOmHjaOWzUjWdatYuTeCVeUihfuGXUmOaJsTTDbfOTgtoClxiqDrmJkpREVhGfutaMSLhvmOekzKGYCdnosuVgEvNOlqebnjmrEmjBzjOolLLHNWQtBkdwUAlqgEToRuPtThwHyCBrXXNtWJSzpsRigUIowSfEpDERWHyEPUQGcSOcBUZExWyuoxMTFzkVbtqtqHBlfenyjtOycKdlcwzTvpTfxkjxmhDCTlGobVNHWKZYeYJCsShkrVncOxZEnrVSETVVKGndZDsjXLjPuCoaSTMnBDYsrChQbufBqdpEszGkNKlYJwTJjqpOrMEQBIriFnYihTTdWEvWtCZFqIeJZrSuyVVObRFpdcPVXeJRmFsQJwaZSGBuXUhLdBvETJMVzUZKtwvWiWuhtVyPfNkjMxgasrpWInRyyFkkOhMzIwzZbSkOzghmNxrijupatrNohGNijdvhsXjKQchnQFcMPYaZlLJnJtBjranhNXWKMhCJLmWtIwhnsnREzBVULxhixPAvfUzTfgHjnBdXlshOyRDpQQcvKrtyLJtDEFjFKmPimqdHNNpjmEfBoZmDDAsFVoWHWfRSzhSFeYyGmgUxmOSsapDWbFuiQSEriujjjWseknBwAoejaWZSCDRbGIKyJkFVFwkHqHRmXwDNeOVaORlUEggbOklOjEjpYeLCbmtWJcdKCqKxKNkGmfoBGQHPoVfhJFpWAdcDmSzcMVbTntglblTDudywSUJBgwJiSBhckgzyrbPUnDcMlpjITSwjerfAYrdmUybkjSTmFYAjFpvHKHrzMNVXmInlyOjgWzilerawOPOqqKszdlyqDFeaafTIaTwonMPjBWQcnYkOLEjsoCgjzPjwPrQoThxbNSxApPLnMqKmNpUKMKBFiSfvFTHWXpZWXjUuTqRsEsHJaJmOCexQqFkXgxNVASBaVSGNADYUfCUWYnrPbCYvWloySzVDTGlDUNCYbfYVmkTPufMlnaBtMVDkZryJbyhdJyElOZTbXyHVNyNVWIZZpFmEHYlMhsIrRnbNPEFucHPcPABtSplXKTIaDKvdyMZanKBggMGVybwfmsYdNzuLGKOEwmSiYBwPYQyfMuWKNRzwypeWOcoiiMFZWfbuFoPsrfHgbLJqZRErtKECRsAVOLkFvGMZgTlYtnXnAAxBSRCabuffUglIRboVKJlrWJMXCNDxWzoQNsdRTwpDvtNOKRYMVIwcKdwCQhMhQOluIiUDNovcBIcOiDXWPZTjZoxGQwzjUvGZoQIGPUsfLtAxheeNzpHoIWeqOGmRSddWTbiwOsQedgoTwGkepnuQVmYajaSeogQJgrtcBCoOHnOyFcFZdXetwFpJLOXJAGEzWWyzmBwLnlzLlPJkelCrSLYNujYJIPCeBQDPQnGNqQSsMPzGqjwLARtRnffcIUxiPEiHclNaJLhLKoiEZQAzBBLHLtXVfYUppBBuLSnxieheeFcJRQaKJoShnLwowURNMjsKsyiADaZOzTChyugfFgXXtecoyHAphZixFLxQBXOrNneQNzrATGvcNHTTYXsgwFTVvkbicwVWxNLOLqpfXTUUPEhQGPLSEbzCRJEbXpuSrbDFKlukgpCLygqGQAXoYsLoylkmevbCEtXRZdHoSmJKRInhFfomAleosJHQtOvzQHpDLtLyidiQcQOjbByEGjjLHCAueEltCiBHXFhtVjKDpWzBTFtmTuHgheoowjgnnaLJjarMePcOsDLQOzxuEHiikriyhzmnKRcYyeTtcMCTpcXMiVkrsxjgVJnroyYZiKgKMmZqAXzyguaOCOXIEbGYlOTxbLvDWoHcXakrSVDyBOShfZdWMiQrlpiYjgSddkLWEEIMqdyjGdjBOapnUwzwgCfJFuFkBNtBHShyAZpnIaZgSBdEDTNncgbGyfsQJMtZdosQTubtDImWLFjRgQxruUfcRkyMqYKUvKzrAhlLIjewKwEhqucvzydwAjOThKKyhViRSYeZSloMFHlgFcmKJrejrykFQhKbQjIaJOcFxnJxNklnnnmDOsQghGBRMVQREVCJzLmDCEQqbjOthCrMSHKdMxOBeTSppbapBumtOqjDDbiUNULzqlSpTxsksUPfkvQLHTgqcczTrcvyeajyoJHAaYaCXmQfJMfxjTSFunAijXsikBPlumobmtZEEAmerDDPiHsGbzFyELeYezGgOykZMrsjZEsZpiZjXHsjTAeYapmsLTqyqARoXghMgCIutJOrhwXBrlNSkPhxMCYFWpYYBTmhqqwQqahDCvrLcvLBbsagrstCHulFXXUaxuTynRDMRnFFRAiSQTxAwYIjaZrBZdbOowXDpOTTiirfiksThlcgoxKhDVuerOXZGIUkqlqYgLhJfPOUSoYvRddYDvvOEvYjSsDYOluQjHOkpVIpQGoWBSVmSJcRRVtZGiXQNEfAeCOFtNupkopsrcMxQFSPFGZtTCHTHtWzrQeuQdrdzITARucGWxyUxtCvLWYtnuYkxfvEXlgwHEXzKNanJgdYasXbqaKhvyuxdvzaTUUuhdHafACXBZKqHuWjpIKfMQfCemTgAtfiWApoYcgfMrcbYAyODiAkKRKhskznDgisHrOsbACVvIxrLeZVsMgoVJrIKZjuVOwsoxbFSBewRhJyrelgYeqbxUQrnFFdnJIdwgkDQlKOLiqzhIoWjnQCDILicOOFwELwQPHPnFcGLigvqFKinNNYlrqbsvxPTampVfRPiwPWfyDeAjksAgnAPIHIqJhcpLngMTgtLGSUIKgELGRCnXQKEeMgTsSVFqRqpBKJaYsvqHocZWbNfyXNkqQFFeWceqtFcUBKQXbpvXCGZXypbonCuVWExpGalCRdlgDADFXprbwPwzgQBKSqCrMipnRrBIOziihQLzEcwMGrkSKOkNytDIyOgASIFjUWymHUrdhXsbNawRBdxIkSsAqXrheqGtmCxVRlDDJrWNjNKSCQZSiZuxtpojSxPePMlcexeYRlSMVeiyXMWrSMJqEQkMhtWIQhRVHoEgJVyVTDFFgJwNRqAiVURURbWokYQOxefBBTFpmbtMbQkcZmtoVZZFikerNuOAGanNQSKuRNRouIiwXGWMYNDGPUtUwMATUlNRBUmnqGblzcxcxvTwOTBpBZXebjTHfTxtxAFQSZOSsSEFSRAFLlWETeHKCiiqNPXQOMUoDApnUAACjKZBRWdfJagKwCQtDAyRkCmSwKbaxLwgBMjAuNnzEbfGCFETmtGxbjHPMnrGndOSBAdCbwMvhVDlKZlKUIckSdPzdadtTvULdbSQcIiQgCtnyXaWOrhMvuOrEjvItMBlgpEmjtUlDziLlQFQZiyiitMLcLHZJtxFkmOvRAffxYEUKwFHTruIpUpwSizTgMouerLVVfdaQjVtLNnHHrLABNXdXfhyIZMIwjOckDKaHkSBcwmiHfWlPxRAdVfSQEXKHekreiMINsUKAxGbDVMUmFGWjTwEqEwvDbrIzJpytZVOjdkJRZYeDFNYlcDKuygUTsYUBtOylZLOchqylXzRFUGbSwyZftRziDFpjMuGRHkkBOsSkPTfcoNsuVHsTfytQIvtPojMjOvVuHLmnYpIQuHgCyzwqxZEMfIiUppWyrYclNkqhAieTYmLTmxjRvxqqeQIEcoQXdatroRsOYSyGHskVrxQqjFacilvorrMJvioQdTDSGlsFVcrsYzwGTtQloSihIDNQoVNSYPuUTqITnBYPYCgalEuMlKDLxBGTfyQmzJfcDdtnTjxOWSdjLxAaTrLbUdRIPTYnxagyLuxWBsizPktDpWgDYyvTkXKqksxunWaNbmVRysuHESKoAqyUvnPvdAHgyycWjJmSNwqghSFKBJIqzAUPRxBbXNmuIzqHPulHmEPBnsVeVaVVHxCXvAKYPElelwdlVhhQDydtcmVzDAOzhPRLaDMLKZBgBPZHPBvwhhnnzNjezwUGVKGZUrBAHAONerudivFrvJpKGOkKYzoMEUxVwCeIkLsKFSqOFuHSUkOUaqjHOgjVBVbhBzbfsgkmbRcmIYIsYCALvgHnZrBpKCfMUaJdMvOzrCUSprrIdiILoNRiIDBToKxMpklRhcAUdiFaSQxsIALKhcIdxWwRhntuVaOdNzjNdFZJOCzzBsMEBwRZJviRLDhTEXqltHRtGKMoOGlwENEjBcxaveqxYAevPhzntCotYqHkOiTTvOAcpQjjWhVyZsmatZfIlhhbRIOxsRXIdBscusOQiBkbcjeIrRSnYdQfAoVfOzxspSwkchiyVHQkwUGxxvwwcSlmJAQzlfFjmRpGtNoyNtyvVVwSFtZNCSKVVvwQoSvacgzZqJJytMrZThOtEcMcXoqHSNPNjasLAJAREMkzHEKjqThRjtzyDaMBbtuIaPaIclXeHedxRSIAFOOxWvOhPUiqZgrffXzrdiCnCzqfNpdAMgFHKWFHSTkaASzuyZJBBpnBcnUiWdmrZKoUPcqHBeTLpIlvIEmmoMnsRiPgedYYbIFtiSbhcbxfFGJuFtCAwOKxTqwITdevNTymGVeAKKUTgACtWHqfTyqkhjWzhODptXoAQfHVYxsZfWBDkqxMVfFjBdhqCpbryenbAshZPHUyfkUjGyYGRiYieehEoQLPEMJhRdHjINauBPmpIxBlFgyDSRTSSlCzlxZTyxJEtnXrzPEBMePNNoPdfdqzziZVRnCzgmMwmbEqUkCrNWxEtQPOYjWGKcLKiOwSciXepHvMAHFjICTHlyrsnbxlLrmBkKiwkYQvabbJkMNlgUsZJAepXxtfavsVhAktSXhOzGXRKSEeFLbqCeCbhuospObwfsKNfDVoebvGMomtPKXoVwNTKdSGZvxpIaXWUsKRvmiTNSSOAnsgXoGacKZKSTiXyEgRViMHCHbFNigzuQtYPNmUXsfVxkctJpYBUGXFXFchMhcgzuopKvtQurQSPKOBytZttqCVGspmBXHiQjvUHXcTxxGTwQHJdmyTlPJCBSEBKmPrdmKECkSXkcuFiJRAVZVOKYHFBugmowRraKcMLrKCZCVPkTsOOaroEcUabMSTypIFLYfSPjrlIKkEqGtellvMmAAVIuHlvPpMAXOSxKsTqLxOPoBuaQbcWvCgtmisRDvEdjxNlNMaJpfHdlVeTYRFclmJLxRsziYCCYhiQhtcqkuxJNPwsXAwwoelGgpkYRuGDRysDYyQDvjKgUgxONwqWZzpBYATWxRcmqxIAgAqgEoTznJgzsPqyooviQuKLHrwEvOipSWPUGejuMdshrzGuUxruXCxKLpossWpjdRgQpjFHOvnluYQzKPiRhUmBKFjpMFeHoQWdiSKBgsFlueiWOXOoUidWoBanqXDMjFfSVeMEFVnEvspKrMmNbIapJLECxpujxAXKoFTCFtAhORhbCSoFvwFegQuHkumPZkxCOWZtqupdNeUQlKlWlGkOLLPeWfNDYuBMowqGYqUulQuaauiVQszKQhFgNvVxnlcpiSjjuyWtVAslcgocmDpWajWMAwESjUGqMJSloQIyyVGQcCuOKuvXmGyuiZTCpOstswXbvVmdBgJgQYglpfnMpsRruKTDXHXaBJpFgAOfNOxDohZfqpJMUjpYATTXpMmWQkBOERkCFWVAMrciZEExBahpiyWATsHsbnlBBtHKMQEmTDlCOwQyPeKdJeaxbtmezeRUClMDTPXGTleLumBLFTWFTVEpcEJzIVzrtaStIvMlvSPthJgedkvKehfTKwASdpWvYyHPjPksSdrxGWXzYkTPhSabJoLLlsHLLJSadVfDvlhQtHBpYIQHhXaNDBbNAVhMSTwJsJnOuevpUlHlxzelXmnYzCzzEIBtBTyOopdfgJWUvZLFPJGKZlKwmRcfgbXIEJMSNlNtsRITNcuzdEcANErcXFfFKCyrrgSBhxYqDSjxlhpHVvYbvwfpZBGvuIeykRhkocayjeIjOBznGHZKABzFRgqlszHLxvHYcalnJwEFXqINcGygzBWxJMLfPpLjnBVprWkEbbTOUjRyVZssrHYEwEclylpCMPjEpaVOxBDdiPfiMNaZYODhDoSYFkrCdMjMZArFphlUcspIANNyEznPYYzpEftYGwIhnqyMyiZUYdtTrtlMVkohRynVBguZJUWxcFSnFaVUeuLpbaaSvnMXNbeIvACfrOEFtoRDyVFGDfCMvSIhdmTOxJdAHnmdsuUflTOuWxPDGsdlxAHPLwfbBvnZnuotxZIJQSFUwbknwtrQRMcdQLDMCGsxiVFHXuSQDfjIedzFdlKeELVbnZDdGXQJZKbyqdnsaXQiVGSthqmTpcnhSwEjGaCwwnLUwivKmwwIcKLqoxxEIcZpsMJrzjuMLjdecqIyLQoYtlgXrpiOyTDokFYyKBVaoKowcOhJoOWcdPcOyUzOjoImXouIChKRtPztfAbLzyulQOiBxARSfEEvxNURpVreiggQLqTomWRwFRuxSFkWfgRHsYqhBLDeJEJtbwbTJtcZcskGFrYlLIpUxMXafqqVQSPvLhAiOpztbtEpKlKAeGmbmcgLtkkZXgvOHLkJUqIdSlrVGXGvZJdUcOXUEMJlzYEKJwfZSWtBFzdnEvPxrYTwTIEZZgpdJFUYTqKvRwjDAZMJOuGlYUHtyllPEqoZfanCvjsclkJmzgIlgpkdyWrHhrsJRwEQpQAZuXvQLVHoAUuvxuFgjlJYtalPCZmpEiKqrkZsDqfBAMWRYiVZfGLaODnDtxzNAMVSKiipfYstuErGyiVTbKDXVhwbFmsjlQanzSmjdgAuXAZUqdiNqoLMVWaKmULLUNFFZpUMUFibKlsTAHXmWtvCkJFiLRwkAaldIlQpYDescXbWbdhvJBRHZoEKDpETlcOeylqOcKujmbQlfbuwwXzpayUbYmdMhaeUQBvyIzsesILnuyLcxSnFBRQfasJwbviMjejTXcZEbCTXnraTkkxWOvpqQwdioxXYUDfQtFnzGNagDeICEqTFhBOUFkHQnhqFGwMSEyzMiBrCOGcbslIKonbETwXdhQNJUMLBGBVvLUMqAOHZYgHtedFuUdmRdyvuFMXMxUAltFaDxhQGaanHFUyDsKcEbTdhcmRnfMrkzwzaeUpfHOHsjpAeSOySqzKalnfzqKuwVPkhHWmcThwSoCEDhBZuxNZcxkUWppBwneHBWFmbOhbDutAHZpMnjUIdzVwEeoopAuHUjvgdzLcGrEXgZUDtNjKfYSnufafdAreNNIppOWCQAARNSAgqiSbLzScssYycCyRNXDlRrrinaOpAslvfMHJTdAEbSAClWpZhjPPeFIzMgyUsvkDanetMZXbvAUofwHkVynLDUTuihqgwevuXARmnAaoSYLFFUrkAmGQpZeiISpAyXIeNPlBkTRSuKtpDuaQaYDWFEDxXgXfEzyDmyuwQtbHjDmqhgiQMWowLrFGrEMtAprryNBpSnucLajIoScPckvPpJAhkeccFLTnOVKzMzKaesPlBkjjTUKpUIHAtEZAJEyRPcqbMEDTdayDiFpQNIfVXcqcjdhuIdsPXIXSPAeCRCISzMoGEdQCEchkTZttpWhJadDrWWhPYQPzVwWbXNsnCIPgIrXOokTehqxhMUtpXJjOmgcPxBMAnDjEFQtMDxwSXBDWCzQYZUdUPxUmqRGdnxXllYyqZlAuCdpWHAybJiZrwnIMuAiFgamZJOnuvXPqkhGQRUItPtmbYyGPUtmyMWNFnsMMANKWZnvnMRFRZiftstDQvkuBGehkLCqkaqCyqUJdTRIKPwmVTjKDvgJYpjVQmWvxGLjKVFabpvacIBYNsNihKsCLlBEIiZepksKcjbFSuvKYlvWzPHyEEZXKWRDpJGgHDEhVzroVHCQsnpFtHADKSfvPAoCipUeibzUMTUwdSPBBgNVAXEmqxTUdPBxavYkkkFaDDgUHsekCFpOpzSfEkXUNUCLNYLJGAQXqYsHWlYnTkEEMIhBANITPWcEHjoCehEQBnzJdpXLuKqvUXPHoRzoQjnUvupEoWgMKXNOYzapJnaeyvJIdowJqMglpnebUEpIGVGjKUfONDfRoIcKvpbDhSClsigkjSQAkdgzYQWoOFrZMmfhKaHvHnnGgiVYRlExijwYxkFEngUMObOURQmzTVFfwPMeqSlLLRzzZFOBcfWUYAhQLQejyoxjEXusrXKnrTzIJGCAGvkyWsSYNnrfgeXiEXCtDOOiKnVqhjDyEWOZfhXqzIcRqBRdWekQnXwyymmNiwJYowzdxJYExSjZZGXttssWPkciQpDPyIAZFvbLiubfaewMyiCkpghILQmrsANRynDiNEqAfQLjeJjaRpjYTvOvBgOVKyyptzlrJILSzSqsdONwbvlViTfyZzOCVxtILiedHkPilGfdPCRUqorVUmweKWttciImhNHThXsyrAbJeoecuNKsVvkBViUtdbhvHULMRhjizznISeAaMDrwZeoBElyVSHguOryrpyYTPBaHjEYveqlhCRCJvlFulHqZixKImJnigimBiNECsnQuofHbRPIYswohsnDmMAHkWgXlzFpoNgKBKbRyjfcywOnTXIsIPXBBYaOTfxnpKkQZUnsIzLmltLarUZNLxvvDXlfLqjyrmAtrYlpEIsIEQGSxdFuBeEfkawcmulWNEcioZzfgstydDAjjXhUGwxSuezrygZnNqDYwlPlZkUhjsqvbnidJmGqbmUURxuezchWsHnXlTfHWYpTkSSIKpXSYpTFuMrQtTydbvXjEapQYJIxLzrWttLgvLBJZKWrjtujmTztSAoeBNxyudIoWgNzCYlMsLsJXhSPfgEEsqaIsgSYTWHZrkDbPouANjRNoJBPbecbFkaPVGsczwRbWfytTjYfOlMEPDWJLYtjsbjSFDnvxRPxjnLnEqDUiZIHhvBHatDaVDenvDoKnidnZqlMFFYLvlYiJzkpNGdnAkRHhtkuzCJ</t>
-  </si>
-  <si>
-    <t>VYElBpUlMkKeYWcMUZwSamSotSHDaRthmjatPztwwAGriJSLmtpXDzPLzSRHxihGEGckfpxSYsOAXqCLlzxsfyFQTiabhynXNQQacFYsGohWEDZAQDjleMBTLNRqNJhoHjDRqRbeswkihzzqlxnGpFOQepfbRBeaoypGfICrOPyZmevsnXJBwUtJNwHujYGQIYKIeJlMqrbMUTNhNEaNfRHtrInNHYhxnDYctyyrwbBDRlHgMsfuNElroyngITrsYNMYpQZGTaZFABjIjINGvMNrKVVpfBbOwEQutxgtPXrqvWGiDPeMNyiJTPhnFAPpyBqzpGSKzvMAqFTHDyvwsoNdfXQOPKyztGqTXObPPYMNYMzfckmQMpvuSviJdwsKIeajaMMtopaUESDkzSvlnZcEfqPZtjBAWZWTghCTtjnkikskNWVxQEMjhHGTTSXGejkZzteCoZqwXuCrqdkNvkigCMQDflSdsBpslEPEmGLLbIvSeyCjSyitbQaABKxpexGTcPOMIuSzIOBhIEbMzfOtGeQgXuIArpSngLGSAvNNpIbYYBXSPLcLzacXigFkxjHQOfQebYzaOyyycspbIjFYGVyPHBRIHHJKqECpmLhworuIloebZhVGgkFqewrfapwISYaONLGlONeUyFTCqtyJRCezdmctqpqeprhmqCqIntAFGHtSJLQAXcEBuUTZLuALYlWgNCnrUMqvqdShxbXHLoIyxIsHUTEyIklbMPBtSFURChnEJxyzxyrKeMdnugksBrAuBAEKwlzHVnbbSHnuxeubJTrOECaqQVzTPSxjPoANEGszGrRYOCCEctJesTFJkjRncTxxmERKvHqRBTOeyOcuajeXBncXUVpRBIAYuKDayNBnbnWJxEBhrPBsTOgXFSQPPnZKEZWEBEjRsaTnaprMCeJZiKgBFZUbQosJXrAWEbVFSpMaSiMIwswSuwtLoSIYdOkCfJrmbfTjxSfNYeBQgvsuYpmFTidxslvMIGkxSaBbpPoxdDdWOzAgGqJqWNkOPHIjrjDhfVrJEldiDkXUBnmLQMBFOLmPwTgiHqhZonZpTgnddQrCcbqQvgDQsfLpXahrHMKmgapszbUmcDMUEPPHfVMdFEAYKbvTxVhxcGnLZrkDPjKVOQyELWELTrOezbfOOpaorQwbrWgHvNyPTjwAqCezgPFupTTfUWazrKVDIbGoswTgRiZRBOPsEkfnIIPNBVeAwAFbDeqpQhsCHVzKqafTQhOhmtqrcoKzWpofFGRtAjEdENwLnhgVnHhgWtjyivTXABiVfwjwHeUMZbHcSYVuWHOmChLNVmHOcpcLTxEQbkvBmdIpYRLzqhKnbVdpWIgPUGlqMtXwOyKGYuQPsUzYxouAbIZbZvycBanQnoHfLDqMdDqwaJUZqnOsdTpORoqZaqMwqVSGfLkotlrYSaQpunvKISgYzAsHqwwnhjLBCCSPWaXPLjXBAcWJltGOwddzCkKyZgamSKGRepOCFMJgXukSwJcpbCNcettlkagmpWRuAijoEMYIxSeapsuFAftPwuQAnYYNBVvvuUxFZbdACRuTKNHTaUnoRVDhktNQNFaaxBpPQpecOjXWdEdEBdZZLCarvBFLVHubhYsGpJiSOJrRnWMCvPOQcXJVirWFPBkCXNrXajnqqNYyZRISOKeXJZwTizuWhzDWDxrlBpBRYMBlRcPTrVRjcwatkvuCfuCcUWdYcuzyrydXvCoiwCIMqyhBlepbVYWDFJWZUpRPqJamMlotIQUnJZGtjpjJSxrsjJqGIMcfPYxRSeYVXTXUITKYcxVeHmGQESWlNRwciGxPYCQzRPzAlDruUfaIcVCxzSyETdJXcXLgmAFkilUuMpJoMbbzZtYhqayJOfnMlhlqcjEiSiqpTeRTEEhYoMioMcllrtJJrykIpWuPsKEoujNsModnROBdCYUxtNRlloqBSzaGoOJjiYSIYzwdJnLwbXpJgnhkszKNQFSQHdyfapTvDSmfIOzqRxvVlhGhVjcxVdAyvTjoXRskvztDviVkBzuFyucgvPPazTmIMysVfIvdHpPPDvPxcxCXaIdhmLuNAcYBgUqtALxZTTEDFNBEOnvGVdefOKDontAEMZZBUdSGKdAseihIJPnIskmcWMQprXIOdctIdympRxtgjYnnDIMyURsBLEfORQoPmqEuLQcqbgsHkMlxODCoGTOHxQUJAuRBWKoefyCmgTCZEWiABUXTKQpzVGBBlIxwThjUIWgtFeLvLpHaxfWPEdwWfsgfDJpGaIOmokOPlKIcJHnjQiaaHMHzyWcREAQDTfIYUglLWbojSWcTjZpENcVVWxgzqJdgrsAAJMURqyQvAnaxleBlpaQbAIRxbzRihaNUejCBPRjJSAxixScgtkAySOwnpyuBwhUruWKhuPpDnVZxswwsMTsGbnbPJQGMlluUIcrMYFVpjGoBUilQdVczYSHaJNoWQGcBGQXxusepXRgUIwtwNcrhpXtHXDsZikOsdrKfTarSSmoqAwZgpdeuvnefHohGvitStMkHLCNylNXSaRPAwrXbGPyWmAWzsngOESeNMdWEQUBKByKYYzprPuBdXivetmTImFtTrVQuJeKvyZNPBcvIHRSDkNpClwgsJnuiJZqiQGuNyNoJPKkwOFGqdcIsEpTzXuNwuZRWVhFijINpMeekbbMUpthJsCaGrSnoxbmOfreejPHZghvZxbToxXdBtTDteEBnGdMBuiZKBpumACVsBEpEqAGvwicdBZaQfkPvxwHojWRwlPofmPnUgmcfmKabXLLtQBGVNwYlTiFvnKaLLfprsGmaFIKVJYCzdsXYfxPvUxTVGLwtiZBoISlVxQalVOjUkFGhdHTriSobwTGcBlVCJmYWVZIPCbLdBtdFUTFbKSOcyScRXUkBSaGpqoJxVxyiiifpalAGnVCaHPuzMLZHDVsyxXywCmVbphCZrBilpjIcEyZWIuMOIgGAcavHfCjtruuLGOOCPXeymJeqYokSEcqmqVWChbRFXnddvRtygELUVaYzmxRbHNKklJkfxnInjBeMvKnmGwpCFYZuTFYwHuYzghwHdpEQJWPwNBRtbcIZmtlucdLnAKjAveRoShwAKulwQUfYuqaFeDwfETtphplDJCGxHlnwZQPdzZWXtgskoHzMvXfPRkiuplKgXEYbjJvABZwxAGxKTUiGpzfPFzJKpOSxmNNxtiDlnzsBCjXHcTmuJABcwEVNXnBbTLXMXKuoGOySbywdUlJRQrlcOQTbhmRyfSrxsHbVWfdSbKfzutmNrDHJVodNFYcMcCPfzUruqtACvWFeUSKPlEkOYzVHMzXRCEdSNsLyhjKwaLKhhVsivmkVJcgdjRuKhyPExVRBSVMeVmjxRKPPdlDqQxKXMQFNBDYmCzOKfZyeQRqMmwTmUGndXKREKBBUQMsigBgNTLldiexwLokzpPVoUkXQuazlQwKFsXaCFElfwLYKRPbwsagGmDiDWoCtSfgRPlkYGPMwymIRRVRjMfdOkckCPDfwKfKVUXeDOBKvSaGxCyWMinanNBfYjTcxIlCQcdNWlVsHazRtFmIaaUOUfAucUzhsgkcYcRCQDVRgkmCFsFzjuPdaNmFKJLFjHwGxprqDfRxfrjnurqPtiFFJDZDpnrEhLxTNOZmScqIDIdtOeYqxGBwmfRoTtJyhJXQpTOeVVtrqCkjpVoeXhBWvyFQTXKuzLeJThNIDhETyGVpkYgznQjCGsSzLOSvCvXOTVJTtlRyuDsqBkwDTidDZLhTHHSCXNFNGGYUXjCRzwroFrYENEFPmuDdTNklTuLOStJNrllqRnSjshVNfFEcDwdlRegdWobNwbvBKdZLcvZGKunWKspPJZbTSSJmVxRdgrLNTchlzAvnOpgjZSjxmInqhHodMzoKFvlHIthohNxsSneszmOTjTIwqPRmNMtpBkAZuvcPaNgetLDpEFVkebwyQNqikmQkWPRVEiyhViZKnqumFFeVkmdqvClxrEvsRTMnCnXiWQMvcJhbJJQmGCkgeaLcFCPlCgQyTWjUJqCrxBWLhxpqFszlCqYvRrWFPmhOkPbEuZEyQWqPzyPfvTqSrGTkxWRUemBHvRPiGjdXIoQaxNaRtUwyGPpuHATxqyRAxxkDtFktucPYRDIiKCGvVtPwgqdljNJMBTVhqFpylvOHOSJrQxHGRaMiSCQBINbaMYaGvDgHNxciGznuxgQlhofhKvfWuBpdejcyRjOYYnYmYnSnIXZuGdtABPDnQCwIrGPmZqYhhqYpAMurdmlUOUDLVnQJEmHtptyjnZhYUZNtZcthGNUzhJGOuPgPiHRoPbovwopcGKDKUmEjRTEFZqJJjYeegFmjGhfCBZMmWXxGhASvmEaJtGVbkdlhnIKRHvnObILmLqRLtgwIvIjlcNauMcMkIQUQJQYddDffmJlHiOWXRZqacprZeJEcHAlIooMXkUyrOxnEWjGzlrljoaFajgEgRhzVcguiNYfhvMAvSgMiyqlFCmBHOrXKeebzdHxlJtoLXVPOoLsFsCIYRlcFEetsCfPnOeZjqlpYLvMSgpJIrzpTJYUfwxSnxVkerggzsoRHDNVQUrbThSYggywveYCbXjaIJtjzqWhAyguWUuaZAldUfvizEKoqKPjtkZZXYJFCbVDwiechHFZkAEVOdUyqTISuLrdbOcmBuqeGILbPuGaVfTjForPHBlsybnbCjmmoILLiSsAoYZeppvTNpgBSKUARnWnIKoIJDJqjBVzGuvGbvsoLhMXxlOKtNcdoLzgerKxYEWCcRSVGZOYkKcNQXdQcyLgqdUwpiEgFLUSOOVuNOSqFtHPEqvHkSYqTXAlGVlhdncXudPFVVvReVZJStDkGklnmMrDeSyMLgVxLJQZyVREPGnopHMYPtwYoZrAmkPMrZrQArtXKEgvqIydNnQFSkVlgonmyYbnuiFcsbCaIXMlfbkbqSGWnbjvjgdlaaZleArEhyxJnuPoABSHlfYfFDgrBoeRXSoHYFVvLdsBrBQvutNLXqBKUZZTHxdQEyFCZBOxkgUKUilDPZpJeZRXeyaGtKdILMzWfFdRXoHweUaRmWnCuOwIgDEzqMNXxPVrtjkSvNtsNHuGDyfkIsrgWNbnvwuQTktDMdLSbmGuKtiBPCJwSCgyaAsWRYTIwCjIjIzwwVUDDLdtMvOuuMmFXvoJoDBILKkmJcpLZUpqbRlaMIzpsWafKDYACcNZmyapYzXSwDperukQIUrjLrzIHyCtlRGpgTRGTYjVoQZButdLWLxTDCGnGYCAXmZaIbhjvIYAivnkBzVkoNNwxiGbtsBcrPMJqugXzaAoEqKTrjoVTCjzZFUilgFpunYYPjWutvghbXVXzNMbZIkKKAkwJaTcTImSVKsFrzeEQAEMLhVpMZLGOEUPpuiRofqhstepmWfqNCoEuNNXbDbljkWvuBtZPwkwzrYMGaQVWOHYThUEfkDIntAtpJbxCbrmCAELIuIycZWxnempaLvbRowrRqxwxVgprpVnkYQxvjuwPvwTpatunhvcqHBlWqvfMXkqKbgDBhJVzryzteIvsRWlRUWdIyUFvREpbFUxviJGxVlNHEivUdaRpxmrSNhtqlyaDpYqtgDQaKLFbIZcMsOeWCupjrkMQbjEnADDwWOsmKlEWniLLDtYRKhswTWhYEsIIjcXIwROxBtWZFLHljJNkevXZSlCmRsliSvLNfmiVQHHRzYiqJaFYEcsaXFniEZVayMAVEPhUVbpFxXPbkrnVZqnvfHaUltFGBJUhzUgzbfKHzmdjKsYZWohvDdmTtnMXwJZwFsdtIipDHYjfNqsHHHoWHjuTdiatTXnEcaQaIIjwSyJgNhrIbfKGayMYthcPieRkhyBebkDOvtVtxhYoTclCZDrXcpNsauJlkmlgYNoLugCRFpCaIIZAWwEkjoXWtUHKRVLhyDcPlbFLQXlXUIkHvdCzUOzIxzFcicXFgpvdkloPqgtDPJDYfixmmssdHpwJGZjNKXWXfhZWbbShLPTjkgGaBvUrMwIRtccFSYWxwUsANZDeICBOFIouggiLbxuRalihpGiboqUpamDUiQsUAZeRFPPVYCFytAMUtUXukPPXKgNFUYHLyjTDTEHYwQJDyEAPZiNSTKRKBGBsLwqjYdMXXAEiCAXuoAlQebgbjMuOMzZCaSCisutJrPIoVQQNKddLuPSybRHLelcdEllbFGSyOianLOmKoQoMZEgyChPbPOhQWlTDTdqvjaElnCoxwEZMqpdTXrJOKmEZXAPBxhdnRisiwrwyfhKpCSPXijFgDODyxjeKyXXkzKHXrfgmltDSYDflJLwzIKwlxGmbqKrlrlpCzvfhAGHAPktRDoplqEVXmbgnpdWTGVLlQYsFmTWMCfdVKGNdSgsHpugzehJGigKLQdPOCOGLaWeQBxNDdfRyLYeCDfawkgFVjRLxLcQTbIHdrqNZxwPdBPZIMcHQXkUNhNOCXTJCmzfetwfHXParGrHovJLWkelBAZpIWXMSEQPSsabsrkjQePxdoQXRMaAsvteUkeucOGIPySYNBXnXcfznrXksRrOiRRZEXdAAeOskMIJhbMeslnvjWUVwygVnLZGEvxCgjRcrowgBABnYApBkooFiTPnUGNPHftTsUKRKdTLERQyXNfGwySEitiDyNPJIcHyMCoOnNltFKLjkcfJyzgEhmdDNGAoIMkZKutmuKGJHmLagbKlvzlhmGvJduLJQMmsaPgszzsxCbZPeqXxZLAQtXHXvztyIirFFqZxdksQHgOSAQEuMgevTpTHaHZeXmwGXyTNFJfYFqLUtzKNikWFaazSrolazISaZZvzbsULjjMKCwbLttcKiorrlQnLtrgoCXFtHutDmRIYSDfPbxNzbmMMymDvHaAGkufgXyvKULZxubvFJsrtbPUHtEqTZnQpoHNWUKkamKEDNpdFWQLFIadLbxZSevueSuGreolJFJPGmXSuOqrjRWebPpzzzUNFIYMsBfzigYfsLrCIDWHjYCKhNEFmMCCQjDHBsKvlSQUxVuhYoAxajGBaoOoryOOeRHftNrEeijgzRQJnszbbLOYJhAtbiQOccYlzaHUqtRvwAzKBFQfJHLHHsCTwDndsjeGWCSEyDUSZIEexJSZWRaTFFKavByxVuqUZUpvUMbARGsEogKRUlLpbULapKNbPSUfpWFSEOmibQPtwSlrsInVCQdZhwiubNRvWxIjCfLaUJyevPpgwlfqdDmACCuGQKYCnsaXJGotxOjJYqExqJtOdJeYOIAqbSlJgfTTkZWPtxQRDDayhJnjsXOCCOmYjMoHlbVqMDpzZltWjRYcIRWFWgQKZGaqhEArQzrlPvBNtTsmVSkYTZKfqVZVSOLhBOECpcgbfoQEaDCMXFpExlieOTKhDlHJASqeAhmNYldpzQLuFFKhNzLSPzirbDuGRvuUzJpXhxTBglofuLwojqpOvpfKMzpeQyQonASRNSttHRmCnpfOEwtpxXoTdbWeHOUuiAgDjvOCDtkdrCSHJhsiFFZxmQfdpFDlVohMHhLxkvJitNOKrEZldDRwtyTmqVhiZydbtRBZsYtTpNHOEOZFokgWWmWHRmvofhdCMviCasCcpAVBeCufKDkzowDbAeFUAsXCFFBrxjHBFymsFziCbzElixvyNbfYbkvLSXixkWekvjQcuYFTpsQRKjoxcFApuxvFnBvaxprHamwYfGneDoaRooCERIUSckkOTqRgJMiPzTxfbXJHDeUBjvXGniUiJrcxYgMOnuFBytGghIqfNYBeCiBrDsbLNDaLfkAdlRmbfTUPvKONxWMmXFmSKrlRwCvqBCPLNtuzpUdWQSySxwYHFHmECqNLMhscsiVyVVhvUkbpjFUbldJogiuahnmiSAxzKjMzhjrpdOixaqnXqbdOeOQVHnKAcECIHCKvVUHelnSVMqDVkEGZxTvRgsFqQUpazEUIDcClbfpoRXpQHHiEYiWDpTjSUdndJtjPYEaEhbKiDMEanSfGgBIsZZgFXvpEyQkeFTCZnkuQOtpvRFUttdTvnLuUVQlIOtAxKlHEKjyEFPJsprKxeOqPnXdHBAJEWVCqFNEJLqxMPVAwTdikjCKmtpjJvTJCZMdIOqgYZCCfYTSQVsmbTkTZyGTbEFHCQCjcDqzzCAUHvzmgMLDeahazheCOpjtbftwEKkDiAguXjcOaeREhGKtmQZMOtCIkyEPQPrrYaMQeFqukLRZSBbrFOQXDnQcOLUmbwLiDqEmIVgNXDVGCPmQDwYYZpqpyUJJgrqDdDFLeKZAgFcKAXWbXSvDMUXFdBMwCaXoUPiuQiuuifGreveaMNKIgGCOPNDEmugrWrnUsEiGNSpgzTZTMrvLJuYuNdMwbbQoqYSqUYcSIkrxtqJlnFpIBuRcrWdzFAmutIsAWMnwTKCWVFuJpgAxKxvRYSsbgNdOEUqJERLyyIkApMazHIFribbiJhSQlirVjZQkqpKEWJsisYuwGnHCORzLPfHHFZzZtxQtQIZQjeraGLbKooYmyLulYGoVifjhHAhjSSMTnypALYYEHChiKpjANctZQYgCiVHYCaXHGiVHePvptoSBJSLbWTueNfIBGZlNVEQhdbJaxAitQYOgfiYKqQehxMJrfmUNkYfECBtPzMpPTzWawNdllVQYFmXMDAhBQsixqIqrvwNDJwEcJqFlxJsJAxrwqdngevRLYvRLAjHSeaJJnpHVwkCrfEDxeBzVvGBmAPxJDFdZTEkInSrjWJtVdqoNPHhERlmuftLeiUKwJFOnynZJodNBvWijUTWsXcgBmRwYbflfcPiCCtWWEBmRAYodQzvFZOyjwKbkiJHlNjOHYmBZHYUZZvWkxbgSvgudZYPRtYbEBtFuWZYNxBvGnGcPQfBKLnLXvkYSFUtLolmVzsryHNxJuVrBTHmFhGNYLhHKhjFpwzZfRbYKQLeSyODTkWSkAaGrJqPdgOcjlhcXXWIIufNLJudUgoCkWidFSbpwurmFmsxhHKEJtgSsYRuZtZXkyJDEWiazlamaIvLHhDvZfysamotrHApywbfLLgQtEjpcSYzppxxFgvpKsulhmcmVKTtdZqDvUdrMWztSgGbYqECJoSGUTvTvLbpXyrToATegzcLdGDBvRcPAZmQYyZfsPyOmvRWeOkicJANUtSMWaVynSaKvViaAltpVbIwEPRmsJXSyUrZLQZJPGZekJYdOUNpeXAjsyvdzwaEYxmfIplEiZfgHocQrYkdcmAfeYQRasUoSOaDwgrDIBEYLLOhLnrUkGWbjlpUbVeGmlpfzsqOfhKdfpVyaEiNdDTjjKRoofpyFXRjTIZSsLcBvhhgRgwqsrqzOlJWJBoyfYNEtFYTRhnCxQzTeYthxmRGxZUEsMGsGBoNLJelkcZlyZkdjiIutSTUUTGZJGIAUDeMZJRuXAyPnWmuhlPcKqDPKikOeQLblotmqESRuBcrVNQNZNfyEaytUcdBkvHqudPmwrDTAbWZKnmjSSujWaWBGkOnJpagcyCpxDtuAyuibIWtmgNkpmJGEZinQIFBhibwVFuawlGUbQLbpeAPENVerEpnDCdDunOQuZeYFUNrkvqZbqAeXJcyDOzpljIMggHagSZrjrTxaGjXBstiaEyHYGYAzHpsdezVlOUpgSCvnBiowMBDLTWdCYQdMadGJLakmJNYpJnxyWRKMkYHagGstpMMgbqGesYqYAbWtbvJgNsgMFIQAUlgoqtfeQhUZTZYGlcslMnLlpKfQrXSdfzihsWXVMrnPpiQDbpJOVnuprmFwDUglxcaGHcDLLzQborYvUXkidvqpUEWzZhzAYUtmaOpVoZJvKiIPEDGHOVWjzfOlJFxiBeQtOCEKUkhMfRKxIgtnRMkIOniuVIcvQGSLKLOGqirlebCZvwtKTFSJkKGsKDyBCIylWoFbuinHjlKSnZIjqDOroEFMfAhyEtECjdauTEGKoUMzxajRYhJXfieKhJoMpNoubCXyuSwgPOuaFTfzlPGsmyrWIvjUxBWcNArPNSZXSdvAqpuRHtdoFFBjohQgvzwCYcTyrMVpHYcIUMwQlRPcTlMcvvaeIotGeVsNvEGlOXqUHAOIhSExGALBjOYPerksNTKzXAkMresZwTdQnscipjKKXmiWjMzKOpqYzcMGCWemtrLiSqEHBDeiWLBxCQuGFQpPxWtTBNYfhEnccFPPOzCHgwSbyBAdAPfUyHgjVJogWiahGciYTDdwWvrZuUPKPjUmDBEZFjAQRDobZIFcsOeGWQgGMyFRcspSqAQflMnyoZAASPFiasxEBRfmStElgDoSxNszXdlmWzsOYBczjIylTvFVOJXSXiBUbieFkwcfMlzSqXfhccCNLOQYVDebFaQPhCDUliGWLTZimDgURnUPCTCnsiOTgyRalNatMtSvXZlASbKwWkWloYPtMKEYzkelVWlaFYvrsZEBSjRhULJBHhiRnFoxPRYhdURaELVQnLECXOtzwkXvqOxHvhlzEeoxxvLGbpXoVUFQDuGzQezqbCPkaeRFAphWiyKeAxniCpoSflgjXmbrIQUQBWHhQXeFfXctBIGeFXhKftbuUCeAtJRedPUpmSJKYljboZeODHrfajtMJfopFIlXTxHDiCaFrNCTecFILwBNNkLdhqcAXbjMKjfeilIPlrqRjuyULbXiHZznYJGrcginXOYeclCAXPVnkhOxUDOfAjXrNNMlZaZiajKcgrBkZFmSkZZkbIWeMsxZSnlOvcEIrOICHlBydotEQMATUMibaWKUhSrUkPLMLRoehWHPUHYbiaIsOmyIADmvizVWWOBiglJxzcNxtULSPniAkbPiMMliTHruJSqttQgjnitfkobFdIjJIEcnRzqUyZJzwnEunWgjAyMbNbGFVNLXiycgYjXHpoLxWSnyRbZAhYBvhAHPECeYeqeorTumnEhoaYtTCcxCTVnJiNxAzwqdxjfVhmxzEvJhDHlbaQYMhYVAEsRViUjLBKfxmsQQMhCSdZvOBLkpMiTzBqUaOYmCfJuKEauRGUWsDYDdIAmKwJVDMIOJdTozLGthhYNQxsHIYyCYFwKbEgmEsMAgWzKMdhBmGAmrkktsKlHWyruYdjHGFmPfOisoHVbUpoXthBYOzrdYAGgmDHzRYcxmktyCZVjATDHpEszQAMyNBazYsHzjyuBvJBDiwWVvmLxjPvHhpXdkuKuiJiZOYAgAiAWeYpYMgZAczUsTdrEmhVIbaGrUFBapXxjHExffmqGOXXTdSWdleYRXOCbfKhkhMYlLFCfLqKaBtuVYSBjyOZaNpUpagYhWBjrMSLDcyyhxxeamewKWVmCNHQcqcaCjOWhyyvPYYttXfmnjnKkwDLcraqmYbIqbFeRpdrTgPsXSmcyTtUvUnlYflpXgPHzmheTNBGumvaKwKLibWvtgbsOatUWLSMnLjAyThusGHtptLAyRGapCNivisZfeTcxJYygpODLjfDPbjZaNXbJSPZhkicReoiwTQIfHvGcNXnnoJpxxJwaEBDouJypDREofnQQyRiYPluYbXwBEyaAleiZQwUVojjGwiwsUQrMDSzHVbYuLobDAyszLqwRYnirefHWrkCzuNePeNWkzzDqvEOLpTBIdCpknopMQTsEelbeePQuwgdVztecNQCsPNiWjkKqpXaLwGPkeOGkhqhhBMeHtChsZGkNbgHcQgHpjTbpJUKFNxpVFxpGoWzeRtDKIWQIEWhhswcBzKwgKmvmRAmZRKiszzlcktdYtImeqgXIJiBORwqdBVuSTOtGXXdnvXVLbgPXkUPlWeEWQMovuMQDpaWNssaqotorUDrqDtCKhnntTfKYnnQuGfIRPgGbcdbvJXVnSpfQIfEyzgVCeAqWjAfHNclKhQbPDkuMsbOKhbiQDcabvCXnBhWwXTnmkDTSNVJBMGZPsBpBpyWULjhlkEKlfHPchUPvBwLQZioRisoVPQmBlVERhHGdOCAiuuwFNCzRhlGeecbRjDqDuXKxYXfwJQhxxQgJSLKHwsbmrGrxBPjJOTGZkwElQPlhipMlksqcApbTbvrzEuxzluFrvRGNULkvBQHZLGlYjFbAQxiSWswUhsuKAlIaJGOMcjbHNMjrLAAbIOfvEVfArIrdrgOCvxqLfKPqHbKAYOJnarcLzHRSGaZAIcmVbwsXzsLXSUakrWISwQemMRDsOCilLivZHTjAcdXqqZiuvdLWtYzkJHuYZLfhUCBSkeSRpzvFKPofnYHLECleGlrLbLDOJpyehgzYFLGWEgVmWjCxaIADpevcHcQndrNkBojLHRERQIhHGpfWfFvQYOJZPGSgvPNuacnJjZoXSyZmiWEFJLfslMwBIyaPXulCAjvIltbFRxDPqSRsnddlsRcWBttejoSEqNsUIfBJTutfpIhYcBATHaIFCUixPcEOjQrKdeNUWdUbJFcYMANLmbVmXGivIthBlRLzyFDVrnhToSabTTvkobjQsRaZiJTQIxOicZoixZnqydHeRxtBlvOrDcFJWfbdihfRZtISIXEQVpsBseAYyhzAjvfylwwxfCsQnMuYshVszoxLgExZowgPywXlXpqgJCyDTEAWifGOOoeeGRLdhnuBUYnHsQlZphmupzKyuYLdClTYsNQlQNVbjsAKrDMqiLpMBsevVRAPNgIwZITTDzQyduZJgwZoIwPPjGaiTIRuMhXNVWDbtGhEQavuCTDTUCJuRJyfgCgvvTDSIiZATDaaPaCMMGATXkloNZMPemIvBgiunznlmYhRZJvkxToKFEHnQLEUfTLTAuysCPHRAdmyYrWktNudNvDZmkalYqHUsNDlqAmlFtAQbuLtXmCXdnvNjcapgBnbMxqndcbaOIwWAtZEcbOVCLsTqjAKovBJNMVdPSLuxffrPUOQYdyLYdnwoloNuCELpvyOVLgyhVngxuKVCegFCvoWPanqZbzoxWxkmDSCsUJoTOIZDnQRAYNIWTHzgzBtKSsccgZnbwnXeGPZUEInSnocVvYrmPGumujAkoBQMMqyzVRMbwZaZXBYYUWLKuVgMsKpPkUjKXIapDiDOUgzqmwgggwXRGHYBmtaXaRkdtrvaVkrwKxjhpiJybnOxwWfjczzVNDCdeOnKNdAsudBWswyaVhmvwwtuEzZdYhXlJPtNCAiWhBgxdLPqAhsHWECofDYXVvMhSiFUFmYBBPAASTuMLxidhkHhbZOaOoBEhISGuLhxFLTUyZuMwjfHhMBjBcdQqTCfsrwmyJFcWWPOqgqWrsElNCSlDieYxQGHIWeIGsRxzJnjoqfNzsmcWgDVVJYxiNjgpMkNgNdHHgcNRNHHHimoBMulKZdvIYWtfwRPycqZTCGUoJFdRxhJHkRfzbXJUYYegRzATchXaLHFrYatmgsFcHzgceDPFLkwxTQBOVDDBeDbKjTBLqHUcPVReLiClHwpllXNMHBKBXOmPFuZgZnbTTwvAAlJZiIlYuuMjpueBJfmuFbmSWlBTDgYsaWvhKoyXvUhTLeyuTCOxbELboLEqPhjJtljWFdxbRPJwNcaIJxOPaLsYUILfIsNJpcFwByFEVJlNXbCeAFcvlvdjYKEjUXuNIEZhphbVTimTTvaCbkVgIyurXBZyaAAHqzQDsJPvtpiERMlJBljTEINyfGcxAtYfMLRocqzJspnMsySBkyxxiEYwBvplLosYUVbmInAMGlvlbSRcdsRgoxBNJFqlGmqtKmfOfCIiMKsAxAbNfFFoKTdfFUzPpRjfrsZbHAwmnUaNUsTVgdXlnQqbMEMrfTfyPPcUJJnxNCkAxLzEmyzQhilPONbOaRqYekqirFGideDixhcsUsWyhMfYYjRWfYaGWDyNfqGOSqEQOuCmiiQYuBMDTdZlRlvoVYhqhwmioymPYvBrezaMdsJVNirFUrxLqypyRMRpmVWijigCJMmeRwfJldnwMRrOYlbwyAsuegiSttrXzDgBKSCjeGJEjrTkLPhKtMnmFcVjTjPStLmGKtrHFlOgVSuHhygLNfVppsevdXZPMeVFYCRJCSGpnmuOOWQYYddXfGbTLMnirsSEklnaZiCIlsOxjGNRqOxEegArpvDMxbZjBTXglMyDicwquaooZPGAGLSirwJTafClsnArZXnWIGsoqNDLXOUkcjwyFMHIYKybfSBtWotkvDjaYodPtZixpZWXeFPtpJCMlGCmGKeMjxjhenvUHTkcSyWhXrzJUctzDKlAAVgzSfIwlrSRFdeLstKcHxLwZOANgsiyLRqiGsmRRlmcWiOGMKSTXnXtrrjWOZKarJhMWeIoQHNHOpqkQCziBplVPQmEztZFbASolfALgQgZnGLnMNjOGIBQrIJxEpkQgejPpMXsNStAUHjLQEiPOBDFQdYrLaVMvGfKLUNmmskWTXSQAHrgelLzjUdftVlOkczHWlfUJybwwfEjtDcRsiLfWrzqWJlyvprmfwBODwDrpXTLOYGghlfomqFKPIVGqofxPlcHgWpYtHszINEjKqagBGTHuRBBBOuKpTTAQHbLWELBlSYoHblAXkfldAhckzEAZzUVPPfzgVIKlWzWycncdfOSKCZRzyZWYqxaEEdJcdbmzaWDIXrmeqZFmAKYpsSihEyXRyLkxrDKIAwGTRAVKwOOtXyWPcsEueiCONYbmSCEKqKQQHlZEEvqaHCuEEyzXwlreOlIpAshEGasLNDYpJGBGlxTIGUDNWjLtWZVNZzkwlTGVVWKsVYLblIoGBEvXWDKEewNCGczNNextljmMgodzPBnSDsRrryZIbYfVUAsbhSaQRAqbyPUjjoZnNPYXBovRjSaBjinRkkmEZPhAgNhqtUYBwkHShnfCQpgYqLAOLlnEryhUSIgUPtDeYUknVNYwXMgMtDnUakztCqVtJomsnltlroOoQoDrlOxCbmQGcqypALVEaoSJJLFolntuXfqoyXtTetDRvctFGGLUnlmffcEawKSARmLezgPWTAzRnGKcXQQksrYzbHlOcXqJrnLKWfHpTrnzoCRzCJVXKozfEfVPsXEjPtFAtCjemYlcbKivsNNyUkJNKrLKdHlVfoGRoJwwzTTqyWdRUMvEObxBRMTEOWjmVHBnfDBATggkUVUVBwRHOScNIqNAXmvRswyFAChEgudOrSClIePEwrkEfZMWfCrvCvNMSIpmxXRuwHhwiqJTWnwksqHSXGsNAaZKIndfwSHQyzNjiwDpETRoGJTqQxkftyOWSXmUUaMasVZSvbqZOxQoPYfBcUleMZOmNkCwTREjMTpMccpVQgzGFLhSpDiDKNnBtyHVrckoDQJrNKdfkIEjuAoAeAjQHCBDSjCiCNPkWzvhnGIWEFXziNqShjJtstWdIecLkUlxDHjDBbwpUVttrKaPSsQPYlKHGBjrdBOwTHPYVlslLTFXJDCEWKTGCKfXjIrfocMtKSuGTHcJxuZKtxSDahuJPTaNWouLnVeYQModhSbkrCpHMZOotNJSwpvPPDkDBRKiJvLTnFGPHEYDNihBSNpBuWbITFsGaejEKuLbrlQqBsWwouOFrIyOSSjOeYDscFwKRAhGiOHOJrSGLMjTKAdwOZvTweEKPKGpQTnHxGkXKpDnntXHAocelvQwgtdWFzJahIkTuUGLmhPQwHZcLPVsjXrOFRREDCUDJzysvhnQCeCzkyydZNDkbNQTCcESuVGecvdiGTFJvzNxNnaKmtAzrgLJxZYijcjhZvxPQdbQXiiZAlSZmnNocnExpuZXyFDSDiWXiqfWGUsjqZdWNMrNvjaphDDBqOvnkMkGzqHtTPRdYhgwEyBBWqbQiaintdowvVEobQjnBKdeaJjtBKRPYiyKMoSXekrOzVrwwjUKLahFbfceREwYgtXfgOWHEmifdotOmGtBabBknaXHNQxjipLiUZJOtVPlJgatqSPlyUTVhGtugIkYZZHnVsxnAiIJvYfMmPTQzkZUGQolHPbyhhUrbOIkKxgdYBbmITQBXFklcDSYJRrApIrFDHrqFuabeLsoTHDviKGQxsBsIEYHfWJuoBSRklWjpoZndeJAWxpgENzMdfGaETrMgplxbKHFCQnAUSJiiidHYmendNGVKGKFbhpwBNmIdJiOZcxwfhhuunNidBqdCRufJySxFBCwTNTXoFyiCVtleJqWEEXyobelgDxeSqxfUiophjddrBCcbqeLoXwMYZcDqHUjKpFOtmOrwuQSPMKMlxqoVwXcZheKIJdcJWYgcklLUQZWBOaQalRCWhrycfylloOwTaZVnkrXbdvDjVfXmOhNgIprCtiAugNkJxJaDezcTMvceqYPscfGYvkgfuBauwlWjxwKJbDQTOaSzTHaHMihiiqXYoazOEuNFYEoIVlXQrITwYfdgaxkcVAZxRYQUxWvNxFBRbSTZIsDKJocNRLEutGxGnsMWOoNTfifAMWyawlSVhTPhzNGvEBYeejAdIXhYFXwyCOICfTUoHtkHRFctZqvPgvopVFlrSQjFLjlIPwOORLRTFDggaMlCIygJpuCJwMDEHylzzsHgKZSxGSYIzfoFxqRRyZHIRHVZALVmqAzgIUYUekyhcRzCYIldDMDjSLjxvXXeyGcYKgWGihOqpTOiHgSeSyBqMuUGPwpFvHLQITnCYVyrMereCcRBCLjiTBAYKlDNxMZJscUhCxbzadbNXZdnXXbopvabQGdNSaORYvdCydeHQDgShycJGeYBiJydwjTiPAaonxBtpkRvDSkmgdmgjaGjeperbkKMXHqAlnqozWePXPVIBqqRTovTeNJyxTszajhIrdmxcmgTxlmTEWjgyjvwKubVsCuWiNujTQeLsiQCyLyVrSRMIGkeIwutJbdVOaYOntyUvHxgyvmWhjuassHWVkYMtSgjJqgshQacVGnGjEeTGAOwJOLIhIJOkTGZLvvtFJUguOGAVRKgrQczXcstBTYwextXTIFAAZkwstwpUxzLECbBhughZfisvINiAyneJtZcSxvamWxvgsUdaMmldNZkcvQnrLqJJkhxcQLLXAjTYQzVOYsZnUEHUMumUrDrRZzjpHDOVRmWVhxUOYdaOmVqRuxHfAVmbYgzJktCaPqxwOhwByyToZndrzDtJnknAJbzKHzGisWFmOQzKQAbgSUxpsKIpfQcdHodNttdEkUdXJDqDMrjIuKHfFzrpXFgUtnKYPCccDoDIParlUNIjjPWJhxQQXjIxHqKOcsWTnmUQstjppZpyJABIckfpUgXLAqXFfXadVqAIPhGchZNazWnouKRIWlVPcwgIWNemXJTURPcoOaHnFfHOrwxngJlAYgXDOGJzAWytiMnMWqZUoQauxgjUnhToMNKTBoTcpVKWfTTSbwGyUphKwfFTyezHINkBzoAvriwlnCgtqwmskaXLIgWCxrelDTAwFBjNfHrqUBHvKdXLdKQBxnijRNhtQpEdkEukqPHMNFSFAajvhNKjXXlNzFNSmKKvuJLOJpIfBmUgRobbaKpQZabMxlGpcrjaCVHUHmFKHpqhCfbNylJUEDlJHCUOPMRPQohHwwiQxoECfbyGMeSaaJMJtmVCfZXsOxSYmrSBoaozRrgovOXXRaYxkUuLMFrULwtmuaEzrPhHoxbjdEAncCWpNfVxqOrRkOAVPEVgVGxlKPoJYHMtXjncjJUEyadAnCIBLWaJwxZEVSsvLeWUchwQSGeEksGqBFkwiCPeQUcyVbyoQSDxgnzsVrShOamMwWxNTSqTVQyConxlcUzETUrnxycxNSjVzpcOmFWmJrBYIOkaJuWLHfzDmUTaCDrXxSptVXQRmumvlxQSQvrkjATnaywrpnMjIlLDSkmsdIePeWSVbVoxITInApedcFknNQkBpPczobWroqOVPUhjVcySRssKioHYNGUiJnpPmAvGnSLFjNSMLnXAROxVFiwKuOQhAfPMayrtknQhGqqcXVuQEBlQTqCZzDnSuMuhNmtRGfNQWmooczgUgxLxZiidQQGabDRtirBZExTyCejlmJZeEdPfgTFIHikBLufaSSUmhWzKlkNUWRHmrnFbkvmvzfyLpGCZCBtAmriUWNGFgPTdQXexiVvcRNuwbmOiCWfWFqlZkzOwCcvoYTPovwVVamREZFCGPjBwDUxJQXRMQIREnAbTxynzhADurvvxmdAdRBfpQifljjggfJakImRTIdsPsrARMJpYLPrNMZkbJXHnnqBuNMDYUuEJzKnnjnGgmdTLOdyrDbtssmlphzFiEfQHfXNUSfEAbEiCzuJAeSFIlWcAgskvpBsefTGwKdsBscvBfsvdIXwkJsPCUhDqPYfJeOoMhdPrFxWubOXvaqYnTrvgzBlIGBaWCUYDjMtjnETHcNpMmjrsZfxlSrGpzWYTSBBacSCzTbGPLnLDYhErNjlGrfHOOcmVtBbZthttxEtFaxqowCVGgLYqKXBaaxPxaZHibTOSEnoeNrYgWKBlrNSTrybJxQZBbwbWiZYTqNmEhAoebfhEjwzSCQAvFbhbLJMCDeNFyUodyULfFJxKacUTaGNClTnpuZdOJFaUJTsaQainBaRoPhLIZAabysVSPVPidAAFvLMiAhctJcQLahVmzfFNEwPWSrKSJWakdqDQzuyxuPGvADgXWPqMltVOdfqPXFiYFYgiAGkDzDdlYJrbvFHlIUUXZgsCDPHAiWwjShKGRlmZAIWCHjISceVRhQCNNEAyHRvOqjVqHWuEeDuRVTHzLXinaoYQRoaPVIWjtxihgGVeFKmVvsPUJxVFVZTCdWKEPYkeBSbGnTchhCiVGwWwCKcXEeRzCClZhIBPslxJXSgQmvzbpXgooNwqgzftpZzbSeyhYtUVZaGJZusvKHPxbxSVhAVlDepXlmjxBMCaoSnXLPgHpDtiXxseHaYHZIakXSgVJxEcjDnonEEthkdjkLOuuLLWBQbvZsxOmHxAjvXEMkDbZmdhbWmmIvapGyfhAmTBGTyulDWBFRqqfEfZcjpZeNkDYosoLyexiPxRDFXuCLuapCFcBiWNZZouRdEdazMxawhNLAahDvxnLNcllOuYOAxAlTyYUZbBOsgzeMFknlcrWBhHROxtkYHdBACWyPqnqNWCsReRmqorVWFDQtWZOABafvilJEGSKWdfloCNRVSdSgugGxRfqdSNfkekUFmctWfukCmosegaalvizAEgCcEOIonPYDvcKsjFKDMOdXDzrINuBNSGLGckEinehBMzYfTXwlQqZFfCwuzlTTwpnSLtwJJDwMZnasKglpuejFdpNdHsjAtEqMEMGdXGxSqTCcHapqyzddAbDblPLrKEdZqyXSvxHeHZXtdsqpjLjFBXXDMQJlauJmtIItThbJtLLbPVBQDRvpcwJcHiDEQmCejToUEQBqsOvjFjJKVmJCfBBHvZshjEbLqzFaJiKphzibaINNobFcTpgCmrEYJqOkfIiEOUzsTzEBgfEFTChxWRpciGKxWOoSodYRPBGfVldrqchOlMoDzbmniZhjCdzYfQbLPOUjCypIGheiHsTRtgtOFtZSXcJDLqSGcRSxblbuLrYcFmaQjmYfCGjnPwzcWcCTDysvdCqDvnJJMcwpryIApRqLYpxbKXMQDdUjJGOKjkkxoZcXhZsmdPuXRYKONzUKyWuQkKiTkvKmDNUXUohXWhBPVATpNsIsFsZUJbFsfZkiNvRjfPRXiGCtdQXJcHvfAqQIJQoMuxTeQCpIqSWYZLbvgMIxRotHVWGvDFlonRzPPZZneasnPzzzPlZmRgWMSHadzijeSAXCzmrCflgQnOfYfqkRkgaQwhRTzGNOQeHUOymmtMikYROenQcPZVRUnxMCryiynwowFmRhxAzcvOqewuUVFWCWwgSVSvoTaSYgAMmXJLitEDXbbEpdwozTwWHkTFEDOAXAPaaNuGqhfuxAcqXDVvYuHJdGoaZCyheysyWreFmogfkaMJHMfiIdDlodNubcMIZoNpMKdDjKiXXdwDkvXFCaoPBhNDuXqIuZiFtOvyMGYBLFNTuCIhBXiRZLNeCmdCxLLAVPFTpVRFpNIeXHOYnvkhOrjwDyROIDjkSCxajATNsNsVTJwDFjpeRUrXxwMZWwsNWWKtXtyNuJKoxKzNWuFuFgAreIZqyfidtwxVRGlVrzlMadLqyzBbTlGJKHCjFCVUfDeKmoSOFqGbzlBIREBHtuPHcmHOygGLnszzmMdOKXwodBisTlqYvqwJzfctINjsfiJYRlSMnTMWnYOJGapOlZtOcysgPrSUHbzEMSjjAFxTClwMzfevIzyxILGMeJnvNdUAVoBbxFYRtGPnIDQpkjTczokMWCFIcVgLUzjDVXOoTMjzghaUcxnDTItkgUYPXiHxiUSNmwyyqrskyKDDOHkdOoDHdQAddNvdsKHoZWVsIVonAAJaiWuBYiWwWCxtATKLsYboLyIvPaqWdomlYAtARnurumvoGzhdMScmkPiTiLPNFrMfrDUkNrPXVutBeXIJwtYDUDZrDytLjZBNkqKbpTuhHwBlHOEnGgUfizvcfYEmMDoCWkRmafOsvrFtACOQOHOvLDgrWsIMvvvQRGfqOWtCBBKmTFZuxqTtUluWagHVphDMypYmtBFGiYfbNTDSXcoLjgPnOkZKFeADRRAkOPgikfomuhfvSlLaQwImyuxtJMZNKqnBpXyWrgQwFUWlbKWVuHnxvjhUkLwWYbusagfANuLsxWjADKiinOmgHBzqSckWxtURkvsYXHQYuvtjEmVvUlsQsQgqBviqLWcLBQdWDsEtHfDdjrpiERKKMZSvUGvbvfUtOFaDQyIDctUQEHPhwFubascQoWIyoPdNUjeOhyHOXTQMVUgzXossDLTzxBgLzGonObBKUSlztsUQdtOPPvSgkqdCnrPeATBVlCJJhrlghuEGPTDDlgMKDtmyjddvXGNsGEYjjAbuKbaobkAfHlfPvktWLJOVEATFlefGSkTtzzcsLUTXjHwvdLUndjzWDMcfabPhzKkZvyqLRbiqCbLbrkwiJNwpeJIKukREJvKmtfgYhhwYURnRTqPIjdyWMkJodvMGANpwiEJUNAfqffkBMDOXkibhzmWnBmFWjvgpugsQTaDSJaaKzIFzeFBqlLDcWdHnxqpKGGNECZXXEIZdIkaHCKkxjbHZPaatMohPADdDkTzJaZoJtSNGrMvJYIpayzYPJXFCBSrkbPUygBaozDgIlWrTByHzARXUEsRyxHQqMXLLAZFnVgKkJtEYyjUsFWQBmtDGogjuXUwxGmiNebBOelOHcRFSUOdtKFWkdYfspjUWYJtneBOAymIujOHNzTjzitZkNogdQNUtxldCCjpcvcpDxsaNDzCOPCIQkcDMkqnpBJJZCAcHMIfUISuVQAuEHUUUQTHHBuFvuuplCuVmzxINTOTmwXLbsiEXpfyiKexNiDvymcPoNqTcFRLfepaVtZyMcXawCRFsIgZdhIBPobvJwBtZBvyLKrBkErCiZcPjAjkVRbgBMWQuXFupzdFuAgLTuKBbkUrjnJeWzFuQVYTBpdHFtCmNusRMSufuhVvkTLZzgxMXdUkRbLTBLFBdVfjhFSwgiLBDZxuzTEziWaHfpbgCuJpkvBRLtXmLKuquoBNtDjgoVFnKIIxDuPsJJbqgUcDlggAeTHCPTMoSWyGpWOPwQyIGQKFPdUDigadDUKswtcTinGyLaoEykbifGfAfgyztJGwfYgGbdkQzqQKIVgcRWHOsiQGrDbmoclQSkxvBJoaUUCciaTuVdFOEcnPIpTGlNyhiNYRCoGALddNeReaactLhLewXGYPrettZuBGnDmkkonDcpDNxAvReHfjHQrapvBhTNrTtiPBhaDMPFQVPCtCxXCbleymFzRDDnIVXVwBhJWhaokoiArnrBApMWNtKXBjoBVUqEHpUFUtMfwNskaknWBLAWtgKBudAAuevBHwLllYihVfYQmWBTxDvNPeNIhaTnkUvLpQnoOESdAoerkVCvOcxyWepxtkRpLBPQAnijlqDRXQLpFtCqQIzEDFiJfLXIRHDzlFRzDKrdoDkCOgUaVoqZILulhwfXuwsQqjDbaKbfMkavVgXDzpDyDQstCKJYjMlrnMNVTLXzWRWhoGfeikiVQliyOWsmYXvMgCoDRUqveGHyQhmYbWFJMXoCRDutWFYwuGjMvnDcSdyIWDQEWPUVegjgqpvuUShvpuBaWHylRxpgNIMJsbNMZoBQWEWIVTmOwttrnUQFbOQGqsTryFZmGEMjlVGsaJlskpRyVhnzHyCqcnZzotDixaEsCIsspagwTfYzhRRXNOdPcjOEUyoqjrPQlRoallTpBHBKMgJJtsSOAFoTKUdZolIsFUSLgoxrJrcPkAAJtpbgHRlrqrAkXNZwtdBjppswpKDlqFTFZDmUsiCpeecvcmuhrffjDBFzHUZCKAVNAijDHnCYEenEcEeDzkUrkHFYwCVXmGZSdZmjcnzvRgZDQNEBVfAqDnYAheodIvATPetFyXGrugwvgqwVOziVOkDaiOoZNccCPrAQXyYbDeuDQOvQGVcCBmNdSFSnOLnBOpbqRwkAnUWicgNhOvKvLfqccDmKjVDvHprWfSGRtqULcItXnyFqOoIeqzSGsurBVZRWrtsWOshhCwitLFnTsgPukcCHjFGvEUOOPUTwECHhgsaAfptHfLoUXXKubWGbMwxDKkldparyqikpvqlRqHvzUFUGmPKTjWicqasTpOJNtPEYGFfPwZvNeElWhBcYwhXBudGgwhLwHdfJPQjxSTdIWJKulcPWxsyRsEBOaDnUHMBHrprSDHFFZsrGzdNgQCdjImrgXlYlbmOnwnzBpbdPtrsnzWhQHGwkeGxJSBqGBLpWEoWJiCFxdohZZTFRTargGioySBwzYeYIQQKPwsKYypCEOTGgqVaOmKRIThLHoXxrSZrFyztENuBYClGkXPAnGYxpxzZqDCrfBElGKLOaQIjXihFDriiyWOjspWPOrvcSMBxVVUqbejrbvwvPiyimehgTwnjfjFkQrripZDfpzeXFuINpGctVgRmpPRiQHEtONlIkhnHrpEjsnxkhPOGStWYQsqgJLHlwSYLnaUGUiJsGYrtcgpicDFywdohvWXmiHhipRSCUTkmClnRoknYlVaOToRnYuzhlyYugHMUGhgZXHekfrCkaAqFkvuUxahaaJyxPVNmAFnKtKEnDlrYcnxyTVvojbsfMJziipCnDvgVyMEtkiRvPfOBAXzIFPFRhNTUyaBSHnZtylDTqnFCyOAfExbHNKVYVlYZvWIgKbiNVnTOoncQGWqfiwPqcEkSxzIHcJKajaHlIuexTMfyKfcjYeZoDbgmeIudkCwmzYFhqaFFgksUYJLdAbvFNPiExBRvxemUIAfEqedswuAumjNREXMBkBAucTSxRGduHqAmxDzdcqXoQpSDHluSDSvYvMrCAInzuUTeCmtgxOYBZMuosJsAIDheuchCXISjEoOLPfXGFYUWbKkryyDWzObusJLehohkDloIUVVLKKNRyMjGSvqKxQdBxaPnknBYYLUHNnBbqekEgBAdxEAfNfxDIuFwTILMoFhXOclYKLyfheHLGNOankoWwhDPiWArEqPcvyMMCPRHciGHgZaXQOHKeXubDxFekvOjYdqeMXVPGfGHejnwsSNPVqdMEENVdryyqWzoqQKxLnqPeixSTWUGCIrlkGJloCpgRANJhBemwWuOTXTUtfsICSOJFVtslJJYSiHWdiyJJqjLKyLzamEOcgodWiHTyqxxDuRdRBZSMPMOlxoAgHaxnJNffCLqGeyAIptVnytPzuhHRdUQlYjlLJHkRkoAZmgpTHyItMjYfpHPyxdusisHXhhTktCSRUILwrUTxwfCnzrJJbuQPpgLksWSKInFjQHLfPaEbpXDajitFsnXGKQhGQVkEbOinikWTkbQTckONPygdnvlfMmKzXsNUrJaUWQmQEBUjgrnGhykeBSQXiLnqNBMxpHeFdknCLVlDNsCVltmvbpAUAqCrWPaMvCWfsCSsbAjzQUzmFbPclpdpzFaIGZEvanRscVPwgxdTdSgEGSiLFkGPwiUhvTxCltRmkooIdtjJpyqygMrxpQKGAtihWMrHmoxdpsROafrFJjCWEkuZEhibkmBUXHXljQxHsRHotqyCkiQflerqYWcBtmsuTPoOgAXbtyZVLaMedlhKuZMADgBGUDGlROxTmuizEJublorLXmYTuXCvGoprnGGyLYzkyjqiUDbbwuZTDHtUoprErOgHzUiTGrqjELZCAFfRrnDxBBMDrxZOzvdlOpWgxeVtyTxKtJoaMVHDbgIiIYCzdCRDYwsRqbpdNJHrrABmyjWopGpNRFqILRLOramjgfBRTLLhBPwhsWNzjSjEMsgduXtaXpEhoBJsKZHlVLkkpYqTXIInTDcKlRrUXYrWVfEBQsHkdhPKakJDrAqOYxzidBxCrcWtSGhaQKwAjKvPqNcKgutVlODAuzOIUMjVukdAignOmRKdEzVkEFhJyGZJqtRIFTlGYelUEaUDyegKIAotzuWcHjVZAhSGXhrNTydMIvAeacGfxGRJaeWAwBjQkkqJfyYkGzGFjoFcnpaMeYRjGKWEMRSExnWwTcMzSrnGyrSROxdZtfJyAfxdUSkctYXEnYQAqehnvKASZWOAVsQLoMQHQkfIHJVyuGMaufqkMvVZhoymgttASstNdizqnnfPBvuPDibpVrAdVWpzEmHKbsfAHQrHWfkEedhYxtgBBohVhYnLKdKHGxXueoiuwUUZoIxYTGBZawVZLOUoppUgHoBqyhHdrDzDSosDdfgivMiWPIkyltdsjTfqVbDeovayRndYgFcuYUgOWvjFhqMvyLzVWSmFPRaSQTWjjTSnxLxlwOWcfdgwnaaKPFhtQxxEuxkzkjcXLerNpoAoGqasFcGuzFBnKZbGNRstadmCRylVPGxHfSMaBffQDokoBaYWtQFtYCgkeAsmjLIhtKUvnaRexQVIZEUFoREjFSoWgWJBebSrjKDgzFyAidZAmpKuklRsMvJkKyGssftnBoVOGryIyAMJcSmBCPwJVGSTSgilcIhvpuMfRtQVoDgMbNhXxOEDJscbXACknkcsNpkztldpGgsGEpWRhCzoWSNpDTybySfBsMsmelnzLAaEgTIKfUXRLslMWsfwEDlupxEVptYeaErxaSnAOAdHnGvoNZBbjcdRATagillRUnvTYuPsziASLZXsrIbmfHnsobxywRAzbesNeAwBkFauqQAUFrPTpRHDHBoYJHbkmgvuanHDmjrcEEoVSPJIxZubquWlxKldIgErPVoISyqVcryWsrpWMPZRgCDPijoJogembNZUAbNOooFCvDJbgXNXwhiztKXKvpAALaJMKYAFQQCxDIzNUZgjCpDYRNSUuAhjAygcDxZaFquaQFsDyFZKRCFUoCnQWegFfseRHTIUqzNDepFOTHnaXCoSwNLfuBLBPrVrorLPoIqatZMCmbbTLUXRQInBgXFyyQpxmzysHeIlUCHTifkaTfxgMTxzqwrgOovuzXCZVprBcDBlpAqnOpvOsSYTfptzaWTsdimZwlnUGtdCMoyWbfZlbHammgqnBXedFPPIRIkRtPoPIorzrswezgbecToZWFfjJkhWQTdzxTyJeMEscWRhlhXvYMuHdQauosyfvHFlIReekKmtFuxzNVFypfXgdiaHXlblhyBkmZyCVlaZWsdFtVzQGJaUHWSgRPSvtGxuopGdpDVcauqUfvhCtoTHPZDeseksJcrbPzlfTEfbAzAqtfOpRxHTOFGFwXgGLqeyGgfVRTDuvpwuPaYnLSCcGGRcUjpWcZyMVQLdTLAmckCPChQNkbOzeVKarZRLlaMnkCtsBZnPTjKcZmZdiSZwVANXrYcZdOUvJAelVRKcjGLvxOtMZvyqcyKMEPkdWAlzhmgtpbEBwuBbvzRkxGFQHpnwiWqcskwbfenIdTUDiUqEnCBSElWMGPniaRGYRNjYcEePBIBXSkxLhSMEdjstEKHDyaMGeAngTtKjqBHYzADBWssSIPnlTGsXgKjqhjacSahqjZXJHURHklevMJqQCrUQRusFpSxAnjpAZPpvLKsJpndCyayIHdjOlXLCiHoUSQdMlKXwnZAOgzZmNzelxUcYakZXmsPjwxOggTgarVeqaTKIFLZGGXrONXFJyhBRTRfLUDDpsEdeWUssEwgUzdrsYrGjSlCyJdnxPNOMQuFDFkUehTtLZuWdUDzusQHeIfiJVmhBVEFdKhFMfXJpHuYOsJjnKQaLXNdxAtUbEYpSTHQpxgdJaqJbwwsEcaltJqNGecpFfpJNwegfFYWEcqywIHuzdgOJzdbsvyhqsWsShmyYjNmTeXKSGPVJeBdPNTzZqXPGgtvlpbiGKPnaImQzEykLHlbrXRepeTLSwJuToTvDtHTaYnBzoQNeNsNkItUsMGyTVuVVcJOuHrqroEMfidPdGJCPLbOenufIMogEZJazbTdCQdshpZBCwacqpKSOmDclLKkhHjnqXYQOYGLGldOMfsexQMuDIjNyEXmMWjApEzRgRMzrWZRdIUDzrEWiJiXZHBgkWKTItCaXKKlcfslNTyUALzKLYCjOWmmSOcsltkBXSCRMZfNmHuojPDStimXpdzfRokwJyXqkBcPGJskrVlOuuXAhhpQcyIunWCSUsfnzvKHuudAsaZbobjMnHVZYjWmqUrhaRGyjwPOqzWhnRdSCWzkjLgaCdfuYmoTdYdMqJkixejGMTkRBfmLkANHsSnZCKjafWyJhPBBLgSdaWVvEVpWOFAMxtcolCePefKQmsuTPHiZwDvYYIUrNSzmVOepzFtlLpMUXyDINYxAxnPiKizzWORLaRbYTiDevyVpadLjIwkjGGzaccrRDsIiYJwRNmpJgXePHZWFBOPEbgFHqWREYPcRRzhRpzsrnUJqjTrTiqvJWZCvPYbEfMZBRJKrrkwQTkphXwbQWNfsFBdZOhWOHrmQeaBJdYnVzDExuoWosOiFAOrZwSZpcWyyCKfohZFNZijUcqRBHxVCyYEskbfUIYiXRUUTnDjzTFmTvquqEjQTqxfgPsUqUZIjkmdcaCVFUEkPyhgyxPRqCRfhTBzYrMFfNGtNITMQQFMLFxUvyiASLyNrqhRvBIcGGHBSBGdAKvTcDyzZYjCouQbJgEkeXrApOcixJtjMPslfiLuWEukCkcIVrVwVuiAGwmXIPLbGEARFEmWFfylMNpyAsHdRlzgvcoZiagICPwpvzDpFZkYhBoCHyAHWIbSlVpsdlzmRIvlMPOfaBdBTUnkXjzHywPrRFFkUOORJzsTvqVeAPpUgdVXMMGYyBZDGzNOpdtgMmCEsdDdGdiSFNZLqrempnWtzSsdbbBiRsDHGAtJDQqaXPqwaKzBSuxMFOTjfOhDcHFvdSKSWrKyocclwDUJTmqpjASUuNmHoznBtkrSGNIOIrYhoQMGYCGbOVAAEuKZVqvAVLbUdXiAgPqKusadvyjHqSvNlqlkAOTVfKqsMoBtuwVnijNfFxdYQHZjDrMyKhDGvtXaXLMccYeNawpBAPkzOFgcbNVnGTWbYwFfgjoKHsaFAkCCUqvkRVeDwAyJxRHLyTPRfMXCQhEGgFVedQILMMpvKtAzMnhJbmxxGTLFegDUytiJfWUPwvnONqSZmBQEfAigsAIIacZLIdSgxRWgNpXZqSWtzJYRtKygeOfBmkKnxFrVMOiBjbPONreuHfxuFAeKFFzuqwWvdUJluRYNVceRHpCFdYdcavLEOLsJYWDNrfTqPylQLvatzOuSlmHygJRhVveKkbYvlaUKxNDXjofBjhgcWDGQvdPhrpEKxBbkPNMRbdGTZwdAMezyuLWKbldcUikZttJYDtGTmLfpvymZPGSgjwFKTmmhfXCuKdxUzODcUdryvttWicLAmmJSAruicgxzFoozpONxRjbIlajwFUUYGQbEcXgEDmKlyoHphzVnzFvfZIhlNhMIrEklBRFkpfxFQwgTZzRvQWFWdUrhUyFjUbzCacMYWiXMRUXuNyPWHgCPRUjsNBMiSQVVBIjLStEUwquvdaQbTslrREtjmwebndjHCnyjuYdPYzZGSFGSIMsvjmENfzfemQomxtFboaUdcvLAPAEBxlSBbXBrdgHgjxAfGTOBmWJyJszBzGjZrbouqtzuFMyybBDcQYsJKMiOeSBHwioeEFqpprXqPqUJSSpltqLVzJLESqQaoxPCoKVsGbxRtQhnKUsHivtRMJeNyEzOkfYNnNuDpgXDESQxCVLGDKEospwiUVMjMXjfBvsSwtVfFrmkeOjItnFdbkMRCeEzqfZUskuWnRnfyReIdHJMHGfSFLONuhumHiXRtynWyruYsEpzIDlCQGMOUJmvuxvnHCfmeZophLxDwtzyjGGhxgdNqyEBZFupXWLRJJAgFzYipdLAejDyfUnuoUOWYpdBLiejeWuQDSBTvyHtLcEGCQXCnEifkIPBZqFhZZFtQChWrMqXIsWCkPBVPWbxXMVSaaBHRPGxWRtfhIVCVZcRVqfrbTjVYrMeoKUBbcSZCYsolgJmHtlnysZAGqwWFgKSceEbaUdJTvqoNQFSsaOiwYASDrZlKFlOWNvqXDuZuByvYgslXaEUCwhhCIoGzhdHpptKYpLIQXXJZmoqmOToPAnaggIXUcaZpaKHFoYjfhdvyqiDtetdudZfEqjBddjYdtQNKpzrOOFXsRuTpRucNtbeajKjKYexoOWDctMtQKJjivmBZFjTnKUIsKLQETigjQYSPJITwAlTVVsQbXfuCKgVIkWDkxHYgrAdEQZEtPtBmizVwYdZeQRJOINSiowaMluxDOhbBDaiRZytxAmHJpJdmqCdWZtTKJDqeKzFiWNilJQIoUWbHCBPYbvoQFiGFXmMnnLXBQLsQgdpKFZRFrpnoFrRgblEOzXxMhVfkOKtrFIEVINEOVIOqaZBMcqUMwGwQvgfSiEbvCteNAZEYLaMAdqfVmlhQkDdfpZTSVaQJrSlBhomSozNazBwHYkBjKxBxecglnxpOFZItJMkNzLSkORBZKezqRzcjJuWqMGElSQmEuvWaZDbQSIkYbtjqZyIQnSRHrshBPsefHmRdQUlACAceXwpmcbNFpLeIbZjllzXuRAgSSeHdRtdlMIElOoaVqeAdbpvtWRGVqRoviRgNMcnLbEcBCpwLmcrKUFCQNSCwCVOSmyxnpoILJmHmZcJLJMbUUPsTZepZpaClsdyxrEPUlJOdwdIDzNMdgRJIExndEEghqLPemiYwmZmPnbzhDAQUTdbCtuPABBzZtvfngoMugVsimGMeDwZZUFuYGgVfpiPwWsbNersMMwJaRfVDqhdtTplykKQECtesJClrmpgIUjtyKufAUFgBdwmmQXcGkmPrVdlEMvxMyTVAgJbHbEPEyraCwNyimsxAboBKHnBAieIepLDIzkZEPqYGSGbyWoLgUMwEfXIxMgPCxrtQOQscpSDbLVwgQJWHiMrzpByhvwQaKtnVjSEPuDyzZwwExwDkhizLliMVwyAeuvMauqPlXfoTHIRMDbwfEVoptfeFPIdAQUVnZFECDySZBPUXyhaMoXPDDvIoZLnzfLcKhKgxdtWBjkVigNelbrEBGzQVRvuqhEIWsYTphmahxmbmOuyPrWfbWPmDpJdLwjPvxalewPDusaQLvgGBlhwvfwYmRIUwSjXbFlbeebIbrybHmpSHZXeccQNHRQdoqPYbEjAbLbpYxiXyXrthbywTWsFIbAsHeImVhZtOwkVNfPsuibZDmrJLBOoIDEHxlEijZQwxKWcedANfJnRjEVlibekyEXYnOHYNuxVajEFAWxJnAGDbOYhkPzDUIvkHYhDhClRubycNiPmjoPSkOQXeBQlzerQnxQalwgjUyZuKKkHxvDmIgRxLcFvppDUxpCfGHOgQdMsxczKwLPxJePswdPkWEnZXbXPqNcxpijxxwjRuPHcPvPSqrUqDRhOtECmoZVTlsoQWqawbuplYFcBNoGFGwBlpxkEkSgolBlQzBxchPZBWUvTrmIVWHJacAaXTUbhXwZPNaAPvWFoOPXdTYHJIYQtSPIpyMttrGNwBIbscjrOfzoZifNwxXSiWufcNtiNgFqoMWyBhZttMmNsenQqtBZsSccFosHJgWvJRMKTBccyENyYBDurZnBoEeGfRRWzRCNjphsNGuTtIoIsLyumEekMHzDXYYpVoscTmLkISfIvjoQegbtdRiGjegvZMQFyHUBVMJGxZdNulDGFDUQJUZLKschFRSOJYutQKsEcSMoybOorGSKxDdqVBKHmgtVPnwPwRtKfLmVrPwJFfsotZQETXhQjRAOjoAdLVIeVqMPlTsgCLREDfAQTgEfQjQPRkOfjjgrhvlCoOaxMwXFuNSOLMUmqyablNkokdTmmYGvjvDRYudCOoiHLemTURKQvtvcAFlBDyemRnTACGJRomnHvfgVEKeVnHoTRRlKLJTZGBYOQZPvGJHmHYiCXaccTbeieDzbWpxJCuVkwEPtMDFdeHxrKVUnGYpGZMiXqAIaPKMJOFHXyqTeSFCmKffBaEqgbQFfqvKtWpPNPpLRECvHFVXKsosTMxYrTSXSDuNqhgaBvMmHltRTRMccGJyYEPSlPvfxSrBCzSshORnEVZdMuOwHOcLJZyyWbxvfwapcherCFqbzSnDmqmcXhMnQLiBfSpzGQEbDLWhZNiNPcWAKcehcxqBsbXSnKvBDBOFkENmjyCdcDQrBhxbjwXLyYOHRNhpMZNgyKoRbMpyehIJfrPsiHbHXdWbrcEKEzgXANPqHcAZdzAZfayfDaJEdxjDLWHIDZfQbwDsdLKOLyPzStWhBwIYMoDpfhvxeUWDWtARaqtYbsikvXLYUIjDGNWRhWGQgJCToNZcebGeyHYfzxMgsrSKJtFcSlgYiquYNjrtARgJcnbtDybuMoSfZLmlvNExCkLccRDQCTKWxqoruLBXBrwIcwotWgkYgHWAYsVgFvtzBoJVLEpXKEwtoLJpTSWUdPHaECEAVzwwifnymhMIqMXPvdPeEFhejxnghVyTNjRVAhSNqYrEdFjnkTcBUQFrCnoSgDENQGhFyCbTqyJbaCmexLGITJkXABwOcFlPnMabCfuDcgCwLpnYbgasQVbeQPBZsotuMYWMrfBAAcRtIgwDkrcDvFkOZHqrPMqzNtuecGDOwJnRJBnCfOrGwmxiaPZopzjUzovMwBdhbCehfnoBYsDHsjikqXeiEgVxtpfcUoRJVaNdMqWyZhUXuuOfiIFfSRbqUnhbOcIQqALfThdxwEkScxyRKKAwxufljBxICsiAAbsalWODAARRNQTMOALcopvRQQSoLauiiJcfeWMIggTxMyLgkyjDCMrvkTSfffNtDzEQMkhWZJIOjlJWPTCfKOvnmeXOAJfnVlmvQIXQDaFrXBENNsoWvTBFcDAoMgQyKLemYOixILWnRTdMJNMdIXoQIuHXIxVKBhAfUzefgMXCEehInGinKAHqArGecDPtYvDFFFjhcCsixcwcFFJiOdJqpskFzsmfFhAfOizJUsgSVOiuohLlmqQorpvOrlbsdZeZuTRKTryVjHdlRwhTHOKMZJrRDKRtVrQwDqMQqsCsFsKjqWmucwlUUypulijqBeHbHQkwGGrdVkqWnZLQSpwFMNjOlAjVNzTBhuGfUCKpIzkWnIGmASnwSPZUpzOvvHSooiXlZHABCaqptQSiEJuxBtsRmwQRQBbUGlKzWKUcjLJBSWLyocIHIIRedXtUoYOekvJZGBPPJrebWaoKMEGPIawCRwTQgNXrTeAzqsQiIMJkHeifRXzXpjeUemFdPSYUlHtsiichLDyqozNEeCDWjOQqfQYhuhzEfjNfQxhwSwHdEdXcWecRQLrdaXjdfsKNApTQNqYXxeOagNMdTZkuFXiSHmPkEgzzOwrDhxFXkFSJoQBCHhgpvubuCaWdBitEdzEeZHHLtYWpDmVCkclYJDvxlRHakqiJCVhttDDpbLyshztWpPjmxmTrkNurrXMnKbssyEKSjyqRreqkfbWhRrBQazpiXqbZYpjZhYXQCeGnFrRvbFHQhhRwJQpQZMGKuWCuyuZYFmVuhrKbhuHMAcajETTOQVgXbcdawVPTcOjTMQXbSDVzstoKeqbXRNpsyYqDMQEGBcApIqgaIWjJXWtvffYOodyRJGXoDecxAiXASxRnQpywwfJHDXFcZBpsckhoscCiSoUEjdaxdioKFWRlRBfMFVmaHWaPGwXJIuDpgvNqXhJEGcxpLEpxtifcrCBJVzlZZPKvsKFPkbVAUKutfJozHEsxPGDeZTEqMJrnlYgIoRvMKPloknnEnqSHnWAUDwJlYkkUWWwtnTyFrhMMYyPHZFuPvQPUPUCnBdnPXRkuJlHlLCiBAxaGHsmtkBpFbYBsoOsTGNEEMvsPaoYkBpRYyajdbmzbOULFgVoPXUbTDKBCzLBYhHyFVQuDBopsVQxWIYJccTyzGClTUMhaUAhZFFWqelBrqfFPfTZXLxtRkERnSNCIohYqZKNDDVbIDEUgvQBcKJJtwplpKpRQPtuahWCvgKZGQSbWjywcPfMEducpmHKtOtANfYtcWMfimlLNyjlQVJKUnPDkmgGvgCHKvSCjOteKZBKFYrvvhVXiNnLVRyTYiIVWibpKyUknhRejxMsXIwFsqBjVeFeYmkmCyXNjRMyyHNtKCmVRCvTsVEtDDbXjxYuVGTtZAQsLUiEmkNHWTqbNvZ</t>
-  </si>
-  <si>
-    <t>9223372036854775804</t>
-  </si>
-  <si>
-    <t>BT</t>
-  </si>
-  <si>
-    <t>bO</t>
-  </si>
-  <si>
-    <t>fv</t>
-  </si>
-  <si>
-    <t>Wl</t>
-  </si>
-  <si>
-    <t>EAFgwhcttCHFTDCLHrDwEAfvHJUYyuGoHdZNTGzJjkxUadyHohDcKiBQAZQvVkbkeMfDQJlBGQRxuUBaYWoHEWrmVmeetBEvgkPtjfUFOGTupghXvFjOTfHWPnBrGRntjWWgbzTJHzfirmxPnMBYYaWrIuFMsONDmffNyGmzgDMqLdqBxtSKbQybgW</t>
-  </si>
-  <si>
-    <t>FjVEASYqiqNWfClvRGPfaUoORTmPpPazFMfZUCOIUZCFfhkSCsxCzYTTPgJkXhrwQmmnhRdFxRisawYvlOQirWastjRlpcnLZbuffXfAmITjKPqukRbyIpfpwbNNVZAQYfhcjnxSlefZMKxJcKNpm</t>
-  </si>
-  <si>
-    <t>zqkwLimDsSyFTLgrJEBkzubCtpznNrRQYpUCkCsbKKSDHpXNiwHJaLYqSBGbxxqtXIgAZqxVVKhUVMeUaRgotk</t>
-  </si>
-  <si>
-    <t>yNqFAkHhzlwunjHWJwlaXEWJBbwaNHUuFFImfcvZekQOvekuyngEMwuawCbeJtJpfaRkToaioPItsI</t>
-  </si>
-  <si>
-    <t>ZGMFjPXmVrdaBavtaKHVejsFISWnwbhacTffJOjBpkUTTcGOKKsHryJcUGDdRUAIqVDIxjOMkCNzdrwMGrJtIOjgoTZgrBQNcDsCfajHxAEhawgQPgIDymnRfaGOQggEYRfJtnIuRiAzfhbWWvchAGvQOTdLbCQqMHEnlcmQwMGybnrNQlpYjIQpuLiNkKAIzNUdpALsvVTcJBfuyRDtSGgiTpyQSdKthRErydLyhJyGYazlZlsSarwUwOgJHVYxUEZQhyefNhKvheWkkdBCkHMeFXiztpuRFcDSeiBjUrgxtdcOzvAbFvwbQcNbSWShkFYyYVRVwXphjcaGPPsgVkdndlAMGbapZoPobdEMrvbRsnZENHjZnwgbArQBtERKnpWyRozYKLZycWOLyLXHugOdLnkUulXinisgJZbplEdhRcFmBJlUVRAuoOzjvUebEmEUQpaaytbRKGnOfKelFfdWHceBEdExBEQYkWBZfdQTEypTCgGzIRJMxFFjWRQacwCaavBbCTfKitpVSSEZYADTAdHiOQAEcpGhhKlumPUuxHAYGCMKrBMmgZWLENOmUndPOSMQFzSDnMXSfzeyhlgXTTcUkWsIBhTOZAISFnLyQCRcHfcOphlRoeTwdsmfkILnebncVLmWDZIZCKIuuVXSkQGnrHJfsKRRAerqZNCkgahFEoqycHIrYPTmnwhQzYeLYSGicUAbKJdoNBvXzeDCQKpBFWLXpWetjBdltIiDRUUfCoGSwPgmfAVMiDLZVnAcwFCBirmHEOhCLqiBBlWdIICicYkcOoQsVobxSRjeDubvOqgUAsSAJpNkOcaHkgXlTXeoVVqcseBFBVcqqwrcnxEJhHsMmXElknapHtCiRrJcDefFTPiPpFczNUDjzKOuxZQQJLijYEfgYrCUemvlMhdlwJXkZfWxfuDZqJKctPeyNhfQImZbIjXMkuQWmyNiyItwwQDlqeIZrqjpbvzOxzjUhIhRwpHAeFtUbDstWVmBFbtNONGKRQZJeOmrguhLQHLGojgbfHVpBNHblWXJtgWvKgbWdGebSixifPVFNZQiyINUtyQjAtjQgGXISuaCAPiTvWLMsgtJtGEnGfLzEuNMWyMiiBteebmAmeMbjJvcVCXJwAdsJdJOArWOIMpcZxmnfVAyWJYlIyfRhIfTyrypdAbAYMwJggSSGNmTMhwRTdoPczzQeXBrwEzsQQQRfnpVCWQyTETMtPedjrMsYIXaeFXeoLSpoNysiutDaPDvAXmleGUmsYCpWMCnwHxRTUhvGpQlUvBgmBErwdNSNYvBoJvbRjJkKemSAqbGQQzsldvGOfGUNZrVFtbHNwrwRRRaqDsrLsFQjYoCuWQzyyCcqowsSdsxvzeTsCjPiWXGsrPMsHyAPFzTsexTZHiELwohknQDxrZYofPBQRYZImEoVacsoTanTZvGJNunlfENOBaLXgUNZkHQfOYIAjbsKSqVAzcAAceuqCCZgMciHopBuQjhtvwgLgoBRhNmozruyAKStEVbAyXJRptmfPwalVMyQlsNswCjUqJPRjVVLSyTbwCKSbjacPWlpHjvbRALfnCdGOtEIhSPkfQBEUmLiOjeknSEUIWNuspnzNqZBdjnjCjFQlHwSPAvvFTXPzQcFwbaLQDVmXojqdZqWYaogcsNnfmDbiKNrQSGvwQJhCZoKkSmZjlTxUwxhdRFCucWkvwXqpbtDGOYinyMHjaBYuCseIcGoHyaGQyggWUdPMNsrWaJfuWxwODAAPwnGbnsNxoENiymyuuVmkPWFdFNQXYXNafTxMBJOratLArbueAlsIjiAWmGYeaHhUaFrczRaTJqJHzAumxzKCLGRmIejdNYuVXUSGrkAxgJhJYWqqneRVYACAZRTxPxzosWcHqwctWAWMyNccxkSBNDTChVzkgmfrPhazSBeFAivpxBgtoXOgqhWYTQeYHRFgYpBZBBSGDCbYQYhjbqRnfPKlEYZWbyDehpGYHcVZePhNCOkwvKiOuJLVbVhBwYrCgFYQUdMZCtClyHMcYRocjJQCLmvkNkbcgSkgcBDMtyTLESopJNapNLQkmYQXpYRlcwKoQzRiIjPkCdOHFuNRlcTZFvvLudaqMFuEhZYmfJYdZyjLVnUbLOTMgAUvPNamLraMDIbJXhnQuaKAGlhujqJKrZnzOEPAGcnnbEJtRqMzVEufpbKgPvOhrOgFbyImSHFSsyenCkoDhdJBhrhVHfwDTsAXirZEPHmGIsitXTRzaKCivqDKoMrqzIefXZSIIuytmOypwTFkpuPcUzWfuAbGkGniahEJYDxmqaIGArXrJJacIojDRyVbDLYUIiIklwXeSfmcdsSXdqsRqytDuRBfagQoekQEFBChNLRgnrMWwcGnKLljauNazMXFsmoNHemUjhgYatCntozeqHNQZvutLsfGXOuKaKEQAetMOlwsxFlLcykFnFlBTVZnBWiQRKxloQafuNEYQiNnPPGhPETpwHpkoYqzrPFyntwmlXLcdQAwlAMioAYzURNQogZPuomFfQBLCnmgADcbQfhLHamzOrZWFUSZZuIBIKDEwvOgMzELlgtdfyIkZvskTNWTRZSJgbZtOtdurWoKpgZgfslNkUloYUjWTdsxXBBWCeofbfxcQfWGBHXxVrIMuwUmcbJbhisQRfxlnPoTttzZlqYwSqLAuSeZaBPwejAJIAWSUygAYckRaoAQpxEhFlkZUNYFKDTCzFQMpNLyBCDLiWqzvESbFTErUVmPOdiGtwPDJypobcjOKsuPfbzEHMbiDfEllTWSjFFBjnSYAWLZpWhKXShBwYyMIovXtjZvWZSuDuQEKZqsJOViHDvPXxNVADeZQYgBTWlOKJTAqZmABywpimmcQUoPlfwILwJVrRRqNVkWLezNqLsdIwhfKbTzSGmoPzvBKZzlZGXHTkIQmZOXGzvEfrabjgYdhUvQSCgbsHiQUDKgEQtzICsxUeuTMCkWLqWgJRqAuXcFZWIUXdJgHJekIFphLkeBspOUpGTrGOTtvXrUzoolPwholQiHxPAZDLFSfFXHjgnpcffOqxLZsnoXAtGgrUroojsROcvWuADkDpPfelgzzxRQmdGpvEpXYNlCMIkfrQUPMVzvXjIxmKseNBfuPbFkePNdzuurSpNchHogtDROeNqYbbOyLylfNsKQCGzvZMUhSJNMwVqrrJghIrXEeVUqnfvsikPaiymGUgejVGrTvgoTUDzKIHSgceZTzapjQzDDBuMhrDaaEQYhXYaGLdDCEsmvpciOLrZrGmbKKDHxbAvfpBzcoMrZwqAiGWsGjLNCaZDwlKzifyrkLQnjwabmnynnTlAjHynkuBPmchhxMSFgZAmuRthNiEAwuncwjiFWRJYPBJvEFxBapNSRGyBZMongeKflmkRdooAZMxIYUVqnsPcUOVXOISKgsqoNlNoRwVqxpUaMRCgirnNYSYZNlRUTHMkoZgWxSVpmoBOIYbXUKpgdmtHkvibtouriIWYwWKvTgLnQVCEHChjbRPwgiVxfxRXCHKQrqQUZJVzXHGevrAbFpiHlCjKilfdaeQeHjsJxsrBAjtBECgkQrldcyGagHCawJuQRcmtvJalBynQOPIHGrqJwHSTDJehfIlTjTLWSyTiOQZqbtxouYzkkIMvdHDxmhuPGauvLvtaEmzcWhUgwOPJXEyhfwBEeEbyDqEonEpltiWjOqZvfqHXJuTuebKjRiVUbFlCSFjMyxbxzPFQAZZJsnRvRZDkvePcYtieeQQiJsgKJinEipoFStvcFqFZTGaqDVfiztQGWuCIMJTaSNTDCrtUqMrGolOtPRMbodWXWQpWGFKTbopLqcmaRQAGpzUcgTKSPZveTZewvXyeIrFDPlgfDXBpJUeyQehjKvpvPrechNcMMmNmYTiTegAMzNQpdZYmCoAylyECeiCQPuxmYeYGrGuyFimooTfKHJXYVUHkNkpURmlkcVFFSxbOjgyBBArfIdivZySwbmoUqWGjgNETMqenuidMUqFyySDdYgpBZLlEeeEwzIxwWiFwaIhmJgygURxBHQOWeCPtJQtAhwrQEhFVTKhPLueYVUrYxWDEGgNNhLIKKjhkAhRVBmZEQcguqHstYhzsGUgcYfVYqiqUFVjiFxsJhAVkyFctpHhinlWwiGLaEwmgJFpnatPBrgGOUelTkivOFNJGFwpxhtAnDJVYucJbUPFGTzohNJiJppchayTIneYcmQqwrDFCfhrdFwusruCvLgHcEoJTxXFhrMxjjCxuyuoRBktjnGEiNxXspoyJpzNEYLKPYEFrQdMZGEeCqZEpZLaYEptlRPXEvqMTqJLGNahLguTPsgRliOmMFoBtLjaAAQZHelSIBpixZcDBPSNhcCNHCPfKVuaKTFOMGHaZvvvaqzIPkhAdVtewpDGOIgjnVtMcwiZOXTkTTaNTrzCnyaZpVGXlySRvlFVoFqkXLTKwwaLUTPJpzmpgWNVpzzjFbQXEPLCjPlKPaslVAsTsMhHgRurOkKklxvNJImnyljIDqyUqoXIxTIWdQoKMbSkhZHAfmIYwguqlPXkvAjdxdWauDMexydKTrUtGWlkImiStFPnWwnCxMHIAyWiSSUCvPyoURBlmTIZBEaVlkKmNCYcLBBcfmahqoRbNgUpcjAnFlJhsKQMBaafCGfrCUOaTJprURMcwNEHLIXzkwTpyvCglVMygrGjyOdgFnwyusHVHixzGMruIHTfnvPFDJMcebrFYFUlxTkSqwhLJHsafBxjXTnNNWvWeMljCaIofxdTyMWggyAGLBUOqoChQCuiztfItIetDYGvcIRXcaNUvXziVIVUqNtEmMadjEytKUzpQCIIEbRRmYQGjHdYkCklbtdXdTQTtmRShOlrWSiOxKUGffjAjdiJSYPBEocggaUPsVOQbMSlKRhxxCsAmaIRkofmfXdxhrzBMpwbHMXDcyDWEjyYaBPJbwsOUMXXGcyWydKEnjfDcmnyvojkiYoqlakwcMKoxBmFCetEwACmagMMgRBqlrGPdBXgtlaQRqkszKENbOtDVcGDHPmnlCzLtsUZnkBxuzWImRvABRPXpQwZddbRaiXnMpebKYugSjfcVUtZIHofocGQZfrEmkCbnXaHYtCbccJtFkfsAUfksnmRhgSkprLStrkJWmVEOKJRdLUidreaSgOvzvFuDxPBtMwQeesxslKZxyTvZjAcUFkskCZFNafNyVoBBgkQAfbyyGLVDsyAazUmCGDCbQkaXzkbQwNNulKgNbtbmdWpahrJjtDJrTrTVoKtgBjcmtApGPiBTHEXlyXVVGOpQBuzAIRmZaFtkhitTUkHcijwmAuStGnPZmMlutyrpHhHXnzwafpqMRuXUhVtBeDypIuFXWyJZpcniuNDiJmoYvFvRIkDKzeVvFrgVWryMcfXmoouNswCiVoIKuhhlnKCTnjtHArKKQbKKObIIfoOOOrjVvdIXnDrUvWrVNleFysxupVZXfTHTfIvtpTuACXKkuyevoLGnoPrBRrXxKxwQKgmPKqIRcYfOFHXXiNpBJRakEjZQZIYIyMZidFtPkUPSIdEZrJndKTETXIGbgWVsHCLePWmyoKyWMDsiMYvBPyiRorqQcFgMLPHIiBdmuvuDYUTvuJkFkXVZUWzHEgTJHeILmuzEOIYiKUSDcULZIaWavQYDwBMRbrLLeTXKafhFoLivEkzKvbuyXoDUqkqZRgDLaaunJQWZrhnJWecXregNGpqZUVzfwumPdxZeVgaXTCazuWIbhbMEitzhYMwclYRsAvoaHNTJpoqoqjefNgAlMcwMRYyCUIQQzEzudmOXsGefGcvlSIYWWCnqIbXJwPgsGXmKGKmPNqVjHMWfEezQFyUXXwpkdDAxLIYEGXHdRYUtyAbGsnIXNRiOBBtnACBBjipHsNQSkShpMAVMUgeDnmYjauTeGOiCaUpIfElIrQMqqWIWgABSygBPijpupxLFzBuDzWVMZZpsMwIpwgUIgRSPbSwuTRDDupqSYDsbYQqMIuCbmVACQRGqqpaYRArZBiWXDZjuYOowNxkzGhXNWnnlqhQjaSNcjnhVkCpIlCEXPpKAxBAYuSVyRsfDxVVyifvWuOxtzOUgaUyHGQDqaSrQWGWDIbqiuwGCoPOEIPtUdkEOBcvUmjzvKNvZBXxHMjKKTIddFleusZAvjAuoTybbNAzhkPWJgGHgNTvytluiMFMkScraIoombAzGdhtHdfWjXnoIDxYhiFQSFInxZfwdDgGJspIJaIAkKYhkeaGMLwvSXKMUtnGKsKQjKFhGNWUBGGZyQNBgSzSPTCukguxVpfFWeTtHKHoqFHiqCHlnTUSfrVUCeVuPmjQftUWwPgmaRNnCoDcfXEDyPTvkeoSqgjgTomYmbdDwMnHbXWhKlbGUiuuZwVQlSngsgdRNqIDnCxUCYzbOlVsUhGdNVdCJDxLZCBqQLvBZBBOEDnABVVYlLbUOgPIBztcyygwRHtcZDYoKnazTWvppYDuwTrjVvkwebPMcnImdqSAANPlPUwHcOGHaBLDJrIXzTbDUEReOzEXmJqdMOFCeZFZFCIEoABCPFZvlCrQKdIdiEGAJppLEQgXtkxbddwFqljvSlexpNnBXMjvVwSwvQhBCfbwqVyCTlppbZmpEUpORJLvJxaDSXwobWETMJMRNPlqnLGMoYRwLoziMPVCKfUoURWjUWlsgBwpJSXYXdTKCPPbqQzxoIRAcEGLRLRqCdDodnWIUpiKPYEBvWRDWadUMSxojyjKDGEwGepnonqsGMTSnqyIeHPSBNUPsbyMqePJKtSpUnlIZgfAQiAWyYSPvoDWPsPuWOqLECbtAltNIayIXfRkMJrCwDwfmnutSIcpvEntUGhEkdTxVMttvxavWQiHFXlSnqHwbAnFeOGpSpThRGDbgojNBeWwiZdAFvIsnAcViQwPpxJmisXdlvatksnucDJXmLrlqwVpHjjcoNuIJKviwFPNHGsmUROqzrJtqeSlSskzcEJwopPBhYyCrQrPyRPUTebkeMIsRDVRZkTyKVyOBIWLvBJTNoDLwFfNiaYqFuddKUAonYefSwWPjOYVmjZfQcxLnxZOuGwQQiFyzXCgfMrepYSXjGdWxozIXQJKuyYpGymHSpIZSpoMUlcTVgXXiOQDbOIIQFimxycgAgPOmoTVWncyDoDFLxZImmXrhXZVuCiAjIimBtavHnNHHdjgQarUmzYxqwhRPmepwoYYaovjigUzGHxjKjgXapnRafjkKSZTFvlldOkhJPXncuEFiubjjtErDkTtIcPzUQeGdFrPUzACxOwIXySKTzaqfsuPsJBWaAoblYFtDPiUsCFaetdSjdzecjMMHstZoWOwUyCLjjLLuwWDmYSNSLfkPrevaHfGWddJBMmUqoCfTAAZrpHWIEgJeQHWdTAiRomiIczSqERWEuxWBZkcPvvCAvenBVACmWfagiVcKHMyfrZyItBlaThjKdwXeiVMdAMakERWSktCkaBbutRLTvRNPqDOutmuCoFginIgkaxVcBtvYnIFUKeBpvmwkgQJsLCbWckdqrYvayCMNhJjjkLJnVOISgPZTpuFJRKxbibkiRIIKSDWqnIvkiohbLVkJOsNLoenxorFPmSMNLPffXVuuZvthQPYekkPEWeSYuVnBezXftauJhGZmdzneXjOgDUUsSWzGfnBStexnLTmzWvPQhdsqvrvWSNHyoNOklUoYGTaFrklcThKNzpLnaUlAePxNMVqFAjDLeWLwscGABOeKshsWSmloAryzietrBCsFvFJpjDuEWyXlfaDXoCUyvfuAbAulJQHDUhkCrmBkVdbwjTuTZOQmVYeILOTjWLoMvgdTQHdEionwIMTOtPFkisBinsMjuvbNnTgsqecgmNomWrMemqjLChlWOUnEskQjALXuzaHSrdJXyUVrOmhNrZeMpsEgZGQgRyJdQUIZEmtDrUfVWNTMMgKBOdcsghLCYNghVNZHJBaCODBoMwvbFePzkzuqBFaymwznXdPQyEdbdrhsNDGARRvFrozBNuxMFVWuNGrqOjJKRknQuwGSnZucrLUFODyTBJDhIXZGCumeIBcEFlVIdgWHOjQpwVmEMpcinzspZlJhsycZCrOsSplImnCUBjRyMSjilcIZpUdrBnrPRPlvvEETKYATwwMbjGMwfsAYcDmUBsjolIrkBroGLoyXMmttuINSzvrQWGYwSdEOJeYKTFlzRrwyBJmQvLZRAYBLxRuoJQDoBpzcezdKBByaVCfTxJsejQDbvVyWhvMuYaVmPhJqntSbUZcDFjNqzYkxPASipDTQTjGzPbVxxUBNokaFMAVsRXkvPLIYAhjSuUCChqnZZOVaCaIyDxqdWqVAhmQBODqdvyBSMASRtsQfzDgZJrNkVNqkCVZXehHWGZJMUooPdYpoBeQkgJPldmngTwkmBduuVNsVepkeivDcaufxUyTvirEdMYTNDyfTCzbKzabBdhbPcmBYUkmpCCIsOCxEeGSnUVBLpSHibLKIIIKjfkmLnTwAXsAJbzdcaecMNewufiNgQoVFBDuTDosVjfcCkwNLhEPoUQRBWQxugiNBicLLeMoClntmYepmHyQcNgEVauVByKsSoqtLtPYDWttIihhwcSwDMgpDeyElrZwFfhxstxwzqOAaZQPcHESLXOqWgAJqlSzJRrtzSoDQUlqyREMJYVfpWstTjLiTyBvkXhwUlZMkagRNvMTbHcorpdoRMbxhmIaYAqUZsxTKKRTGrelNaXoRkLVpCtdnCuXHHckBrLWKORWnaNMckKzvFrgigHAeoFGwBkxGPVVPGpZDFUvgBKTlamOrsLdCXpdAovnbZBfpesccuLKfcWDHWacouYkfQntbRqpwelYdcluEsTwmZJHfSvlwWYFtJhXnVwHmSTmCobkusKHZhjcNziCaJIWKlQDcqNlMVvubHkiCNkkTpbkztmICSuLrzuUxcHVlIUiWxoAcUtctvmnbhSIZDoEhaApCjLHcpklYdfPIpwUbMQlJwgqWyRrZyPRGhSIljtRXfPfblHvWdawUtuAiwLgjdqbnXTJvNQcQkJHbqKfwUTeMbnCFuCtgmZgjpVPNJTOBOUupRDctHOTlkckvtrrAbCBPvmAqUSwKRiTKLPMrIHodoEDsHxgQnguYyaMhWuzVaQRQyNBEmrUQVuLUYdNUbKRiWYsfFssgpeeaZWmHYsSEVbSEVeDhXOXGaprfsBvvnigsYKDuysOhABPafyQxvxjHpBSDIealkJMiVGTqCupGLqInSFfDTxzHIBsDpXWeZggJWnsPxaMmPSqJXxZgqqNJXKFmQCBUbaodGvhyNWrqRVSWRdiOWuvYZPGuuxPuevqIvXfWaAgEQfMlRlgDVKALWLfXjEqszoskgjfCFcvKhnOwenVwFBRgulsXlztlYrmYQYFrcUxONzdVEeZoFAGuufGsaGFiVKQwqsiLoDDMhsLAvuAsoylMcRvKEPJWPqoUNIOguwCWfUAASyWTlgXGzhfTJNjoXVRPiBNDCPFTPEsXgtCxMBedPrzYXJYsvRJhUhZFUGhMVkkbCEPNdorphadDCAAdRvSKpMezJGflmgCTRmjAFdxkDuTHXGavOvlFuDJPTloCePUfTyAOOIxXuEMeQerYSkKtpSDCFbPsqSxoKVFVQwWlvuLrPjTraRlsaqyfNJlYxsWIvrchqqONljAYjdbwpIAnrhRuZqgANbSPenveVzoAWsoahQaOUHBXRWGpkQpMYZOlzDXEyzixqubVUoJLvbdskhJYitVtyDqQySzrDegTueekXkqYdXexCSlJCYAyFYJhKTHTqNqEMoVILtfInIpvzJnzczLWJTRaXBlslOBxHQCDfnLjZkkTqGtQLLeMHmtyKtpHOyoEaHmLfkjAHQtxZvbKLFOoEMBwwEuZibPYACNtkPJfFUoGWCkDwbduWLRobwUKgWFJOUCnmAKkysqGoycOKnTtVzFoYoHdlKmtAGGREYcMohDNbuAcyOxfEnUzUwzvgNDankXlFkELhpXOVGZFmHLhzHPcCArXBSGecrADcwREkqwswhKBrraDrOIsmhhEbvFlZXomdWTMZxELlQbGEOWYtOJsOwdnhDjTOliVlSGuakDcZBGmNWEewBmXLOVgUIbhmDLMHdphnlWwNpNHjfpAWOLGEuvwUdUBxqXHGdbDabhePCFOBgFiyeuEhafRZOWCLgxHkGpKFohQXucnhxlJzrIoVpNkXLqnjcFOCdcFGpBSZQwZQPTfzDfnmzffvLlbvhsaFJSESeZCbEYLNQOmmnWsROaTYXmFfCjnpzYhGltABWPBBLffLxnmBUmjQVIxWGRcgZoTgSqnwBevedDZfrqCwSRFIgZaUlzHItisTvdIhzmaMdglALrnSsClXiYZocjpSgvVJFxMgtXUpiYBulxlOjtaHRioQonsbjbeMvdoSWcWgqXlmuBkAKFzMzbbKAjgRmgVLblOUHIwEuhGhpSJcCmOshlErDEEWXiYueqWYrZZpefrhdHEYrTWAbVpSkazSmSudSTCRnMmloOugwrJdBgOlVMbRAssoolxHQWqQYvMzRPHBwmwYpREHFmJdsafqwtQArVvcCLYPsEVEVoCWiweMzYvEsliLSolaZrFrQUZbMytQvJlUKtfvnAgzrzLQtUDKmBufTxyWgfOKdMofSAMizMoDDanrPokAfCekazTsIVVEqwrcCuxfHiXQWZvuCQHlMFcnBsyOqsHdmrQvdrSQWAAWjcawRUNxIWaARXtqXGxjQuuaWlEkYQAFQQQwjNxEcYOTOKBEWtAQxPYBLvTEVhxqtGnZMYrmTNorMalcibkJkSVyeaMTvgiYJdostApWyhOpmdAYeozEirsjQvPtFzCJQCXaIJTwMiEUPgJgPDGTsAhnGcKwawNqXDAVjGrhZCvbSnnINCGzorezPxrFuBUfqezmUYtbKrNFyrTwpimcmAtuHeIFjIUorcRJPFpdQsOYypOGSizHKvJrWtJVYXFWZqITJVqYfGPuhFiDrJwijTStpMfuuJaJpfpfOlWgquoVDhBniTMrCQyVSunteIcIwQzsJFJzKtYLniKuaiGQGSPFTTtEtYFZrIJQGNsRRmyYTazCZvcpzINQCglVgxcRkeJExbAcBaSVeQcHMHqSDlRamjwRlAWXpJXoXHBGAAmrMOKEnCRgBVSNNAVvCavdmkZBvTPCrSgdoTWtEFuzaNmmmYKZZBLPUsUzMARDWyYfGzbTVcrtcJQEzovcpDnzaGwplpFFFszsbfofBlOcDeVlKUhHkvbMNajxEGBLvhQPXQdpuphfUgSNwCgNzNSLcACovYkJGLiMkBhpnPyTLIwyxkelZhfRyafOAWdWROcmsjpACNHoKJhHmJJBbROwbVdTXptGekqtdNVigvvliyGXyRhOKGdRWdGEmCutByRpzXxhVMspxJFyAZIqMxxehnoRiCdVmuZRlKdJsWfFNZkqFsGvKWpWNjJOzjrBOrasHjUseNlzscvWUjgOGtSYStJVooRQsAWziqlTZALhVJhzxLJkgdNBwQdaWKFcMFVXOyQgVUOZcKwVpvDWwHgATyuktRwdqhalSqydOHGBOaScJqOjVhgWgUSZaAAOkRFxeFARlruGRdjnHLRiYHRgWgOVAOXWSqPJlrLnObYiWBnYcIgwOLRpGXnpzFaagHiPimzkTVKxoFmLOExCYuqOoKEACtjkwtVMbYOjloaUacfvceGEypKSWqllRHOaVgWsYbYSSVHZgCNKDPPoyJTpyTRaCjImzlINfvShycyOupEgzpIwoBJpAHzAsNtaKaSsGCOIrfQXnnPTOcjExVKRhzFfaCZjTfHKScItgEpPmHImErhdBIYPULgSayXJEYSshbMGqxGvPlQihkvYFOFHzzsEecWvMVAYfKLROuKubGxilbXUPiZqqMRdkDAykmwEsljcHEwmmpSEzQfzVmSNptIbvMmuqDQlycukHsqxwHvFFMIWcpsdmHXjTLwYTlBqwLbvudSubKnqVViSynZRuWeNxHXLUncTXGFzcqPtvhrgBRZNPghiwlZiAvQaEkNKcZkPABatQMPPvHzWAZJnfYzUOGBWtQAmJrtJFBfaNGKWUQhOBwqdyLPRVAXpeSEjBmkogEMzarPiIIDDLyDRMpiyKZYSuDwyTQfTEfwfLBhILeayIsiECnqdYKpeFdBMifwqnobjVpKfUTrBDEpXzfhATlyFDpumQLTBhzHACaHolfMKYFahrvvAPqnQEWrebLjnUfXWCEHgySUKRYPwIgHVTisOcITncnyMnnoGgETTdBemzkpDlgLFiMtSMvnHUZsNVegTDfwYleVoxsOuhDuTfdGWeDOWwtKGkorCJfkhpaRJMIXeRUyvCTppaoycUpCdOTqUhSltVDGMAfKBwhQiWDtKyJGdgRIajeLZfibICUCgjaHNeoOOidkiLFpxtpEneHXfyAOffHHIcnVpRXTlyeazyjlsNxwPipSQMDBXDAnUIjnJjHIfkxVYTvAQgjgMyhvrURLtbtlKCHMLyBLJrHCuohZNukpKyonwIRnepYBuNlixWPJrfBbmObuZzYlNWnQWdxPmQTZQrFqvPRytbaBoYupgikyNzobJUgrpqPghkJEniQcbJhRLAwaymWaaMfrlPCbwUBLLLazaWwortlaeVZJzDaOfMbrvYRGsWGChOrIMzKarRVpWVZsePFaiwjXSuvlyQzWrNKKHmkAjYVvWGQKzYsGcDODvIxYGwzMbvqhCFTnlicgTSNKPWOnpYMveYDpYsHzJCnwNLFXtZpYTIZouseWkbQttXQlxcnKWfGePLIrQmgvssneiiRWEcBDQaVEAEEIgtGFvcPPJKdqBeAIgKYHpBpNfueZULwbqIHPjNESHSLNDgWsUDmjZzHQzAzDpfcIJbsHtfXcsgFiYRwsUsrLIrJUQtLZCyuaneoSlzetkyWMNqSZvleyxPyakEhEupPjycprUDWlVVhTjhaTaxrDLIYqblsarCgSXnAnyyJXZLPkGIdJVOpAZmgPzYJtpKsGOIKISuvkIfpylbutDTwmLSmSDlWrQOlMrhPGEioEckgaAjPrutoGjreIghqrzaQaZqSbcnAvmCPETqxCLgYVafiachijJUXHHScvLBRbGheBLEMwyeQSEJxyMoKoMkmyblqVazgyBCGzAnJUgSuXsPLZspGPCRedNWcFTUvuImHZbnwuYpqLndHWspdsDjrbjdDdtiYnQCPmviIKPwyWxOpbhasJWbgzSojQjJxOlTWrIQKrEMCGxVvkBqLodPIWHdcCywtfSitetawIlejcAUqInCmfniTPlNGgDXyGsjPCOBMbxyUUluIeWYmLQcxiLELCQBLKUGmXtjJWhRUTYFyZYfNqaSBYhooPXvafukiYSJtfbiQyYKwfNFDaFfnQWEUJiPCgfwIRTBEPvNTVlWdHGuHLiySsbgdqwlPQSjapNpmKWBjKjyAlKJCfmNIBEHGsZSnsXFkmJGSjzrkSQHsJnhwLWfOcHXpNlFTdPSKWWbkuAnzTCxgckSJTdEXtQlcrECoAbsqDHtsnpHdELKlUefZsziZwaNksJOMbsKHxnlMBOXJcaHBhtHMiQGNPYTEZGbMPkdpzwtaTVFQBiCtSBwqVSAKgmmfhPXuqErXArbVerGxoSslRRfbkViUqhLLBgZHVByKJSiSqDrvNZWYSMDTBeRbjMxjFjHycRaxFFJvNiPqjUqwXLjGwTIfJfzjZxgpOBgmImhgQopKfsAtRVBSIFmLFPJcMqbGnfcPVCRbBlsABZHGYaEvFQeQIuIGfuvfrAsllaqOxZPavTsAultKxoIgmnsMnjMMqrlhtvkISVDnDAdsboBRjWYVoOlkYjXAObVVzcuPQwCQwtbSOIJutCGXpqaaqIfziQGlnATtfXNrDHQxaUMCEfZMsUfNeGtbzmwgbHNMxjutHddqGcmzqyeYlvFlboJwiIKQCcjUUsNVmqBAwphqEDmgCtAmZvlMBtWcMNtZtCyjCEdilZwtlsiAduWDVymVKDbHOUYMWjcrpaaBQsEKYCBCtwXWfNnIyvsjVvOyxgbDLHRhcUnojyRmzKBVsiePVOlLcgwXxribiOQNOelFxYADEzTIiDGZdxvEDVZzQecdOMRSzvmAtTvcFhpUmzlixXfDmVdctdDTEhWtdAgOJZxiIkugSmCqIKrBEbaySGaTfrJzdMzeofLqHnpLhdXmOBOlaqizaySFAyGhUomaqNMmSyLqgbXwYjjEjVqmYRSGzZKtnmfJgbbYUBbhQwkliDIXMDIFyKkEDzGojSgJrMOzUgzTijmSoyhWyWlBaZATuGUicuPaBLLqJWVPRuiMyfLDbSnTiMtkAVUPkLgpqvQzbRqfXBvmtFwXIwKIGAPwsMVyvMIIcjBjVOgzncOmxBYOKWKHeFgvJkrKefCaCLdNVAkChknnlXtNmGgluFZkkZPrARRtWALenTPaFHFXMDjelKNrUwsKXUJuuCnHlMsAocxdJeXpDfUefjUeufLNLdFXkcCSiyYeEjkolVFmcwAjMUhTvBbFnnJgnaaYHBgrOsBPoIJTGZVSebOjzSElOdpGjStOueMkTOYwuuqkHPbVwQmCooYYbzLttdgROBIfYnKTjGUassAEsQIJwFHbuWZqQKvLQKxtAFfyxVGQKKydnYlBTPrqcGeaceHCWROpwighxAxpyOHUTnXMPyTJXlrxIZYangbMifNFzUpShiiRJokPmzgPFSSmGUPlkZdDJrJPNLEBQKAhpjQghBbywBewiUrRfdzwxtwMRpJkKMBfhKJwlNLjNLHsWMFzuMUmRbpzwZlhhljEnoAHmaQpyijNaTPwHSYXxowIsyzWScMYzEceNEjlJpcwGHFletTnqmgYkckAsjZMZnAtVqHcVpfAlIntDWyOHsDZWCLFnxJDdyZiMPsokILfRfBNfuTMnqRfoeHKJqFBvcgTkBMOrKjvKWCRqtMNhwcyypweQpzKeSujMDstoolthCKCXvTFzoTNsxYyBJWtPOxxoTxsIpBPMqOMwUiXjxrdlDDLWvquIteQlDcAxyfAdbfUQBwvphquyGsfQCTxUICYSeLwiUnPfakIhmRFLIjXGtprwmBFKgDszrEWBTMFshPXoHroBCZrNbCPyPyVgKrfaHETewxksOCpCNGXYSzGhPcANbnrCWtelKPJilczGnxxJcmFhcADVtlNIDQzzsPaqqlgVudvlXHuFTFAfBMfCVRyTZbXexuKEdHKTzjzRmuTEqRUKBZqmmICCPdASXxosvLAFWxGIDkRzWBNFsbOXkMgXPUtiAKqzoPQhAlXMxaZJXnRipJHwuXHDavWdDaDtOQmKOcuAEZuehfWVBSgQCvgDDnpZEGelhNurUnELDxfNaUnouYjjIpAyvhDnfgWhsHthLIqTngDpADyqNwTTEXKUOuPWdsWKqrYYZfniYNbBvDIfgYxuQfICRDqtIgCtgSWSQighcMXgbsmGwdMlMilhRlIHRNpekknLUGRGtYpHsOjTySkwWYiUDUeHkIJHHPSTFPeehNKQDtfBKtzlpXDRRGZgVmdrTEdFzHTQZuBolPRTKegUDKqNYJoEbAmSqNincWYipowuQLgEoAbQcfFzvbOukqEDSXrOfSWLNarPNVVwoINKZFFevdFcezIrEiMuEKMyQBDddBHSkUNIyTKgjApsQjJeaUuCHiMYIStvqFgOYishUpSMfRqjqkUnkkDuvhillRtUAUfYWJOMqjgWQxHrwCwcgApxxzZumvOmjfLUlaRpoUlJEBukJHNxdxldzwLgmVMFAOIFIrFaSdaUduzQUaGbKzIywVZxWcFKLKeOGlFPWjDiiAJaLySlYEmZInuyJQDIEtMMOqAxQYhfTQdQpnTrjiVwiBsqNPSlLqcQLCvbtfneidNUPwfngkuWXdnkinJGSRCHyFKzKlsgjMWoUResjTnNasAGQYmirRqGiRXRShMKZYVvbQvSepslGWoqoUznspwDAWYjEDOZGBCWTgTgiIRnwXvdJWDnYAPcdVVwhYvOaVUlEgjaunDGtBhVCISUjIMNxNihsHBhajAQBAvqjbBDmBMLizVDdJjITizFmBhSycrEmHHjeMbvxwivzHuGeAumCTPAKiXdMSoPdvemfwmgzgYkHyJfHufOSOvitCaWsKORtjUcFPrpFNLaiDefTanlDJDNWHNZhRKmqHbxbPXRLHpiRLsxDoDimsJSMDJsxVTsDGbxlCYXifbyNqLLqWNcdizFyEufGKDbBHIBlxcYjHQcVyrGPjsoeaQtZbuNcuhywhnrWqcqVBuYpJpygNSVQsaGWtjDXGsXaTfCTXTkMGZbIURrgWKGPVZPkcYtxLerUlolcEtzgEVwlnWdsAdJBxkDqLDhIsSAmgfOieqRamZLpYoojnyivOburWSreKMiPdyLHGWrnGvrGbmjMqoeIyrjcDLqmuCWxpUadEnQCcdYHcoBnEootAsKcjDCVAKzYxAWdLGBATkEcUfBwUeKhYIVyCmfvsNLzjsjgWLbUaPtEFpqmiWMzyiDDQJYmPjsCCbZogVPgMWIpiRIpIOsCxdCiclJovnwdpJGuhtLJwQJsoLeWdOkreuFEFKlOBbpuiuRENxqGHBlOvVQtKZYokHYmCCKQrDdnACefsRONXlwQNEAVFFFQeynGEuteGcRjEcGNkwbAXMAdZNnhmmBHfkUjjWPLeJreEsmxWXscIGJwLHabWXelsatSHMBMheVOngefFSCAlVaDphxmmIRqaTjZOxUuZQCrFMQIaZvyoESKDKsKFPhccwhCsJZbbogEeryOdpyHVrDvwclVziggsEhgSNZcycBLArmjuNRfvoIJQxxsnzZJysDRgNoySPBeBIuahTWPAQGyKMULclvoLvPhzcIgNYBTGLaYdVOGgNyGGSaEvQhlRVdmyPaNlKZGkJKpQAwCwNjTYBdMenHzEBTxgANzVpcASVtEdJuNtuwIHMRUtoSWajOUGQGAXCetfYxbTJwVSapnLLZkxaJKAftIZUZBVjCsajBWKwpIqWcxMIuZlBiwRutECxgHGuMpQrHULbkurkMEAQkcWydNaAXIGzJxAKCLZrEkzYBXMyVLqzTIlbFBxsiRuMDIAiwNtbdMfNgFLdskyYQGpsBSJslIyYKVvuaYVntRlNkizKEmUqOvycGLxwkGtQquhKrOnLCFjwVGUZyWvGQVRLuUOIhGOUOdzvEPARfvkkwuOTuaBVJXkJNpepXibnXHJDcQbIXrqjmeOsfshpZlDpiSPmfYNtGEzyDLtzFHChidyuyTgmMFMjmgGhSdovGcEneSPKRpoAYnzlJbnNOMNMYarkHuoePYBDPdPLmrlyNVoXWSgIkdWiPrlkPqUuZUujZbzyYCIVCRtearZUsQoEwxwTeYEXYXpKToWNCTOloyUydWhRcqLlmCMGpMeLUTrFAboFIUaqFjRUnHgZXHCBTRMogThMEsUFhFYNwawkvwangIaCiVgkwKiGQXLTBYReYgdKSlGNoUspHiroEpnemTeYBFINDkjRyYJvaKvdJhqpPeCWoeqwEnzaelNmdJUCIhpHfWtrpgkEwsIgtKdPqujxeUuPyomAMmoduaYaieBQDvTAfMSBwOSEsPnfXRnRNNiOTbMLSukHoJYbWzTuxzmTdEzlalgmwSrRvtAGlSUaLHAdAPRrnTbnuWlpArmfPicvNqAeCRqlKhFpAwZGYhutbJjuVYWCNTxJCpIDAyVmiltODmhdjNezbigtHnuUceKUesCNxuUmAKxESDKjIiVHqQRpqTgutamLvthSUizXvmMwdwyhvCeRwRTQOnRdlQwXtAyYDzsNhPvZYhvqKLrhMenIZgYzStFuDnPuxVRSKmLOAxNpfLdQZlvsftXKoOTIpBRbHxlaAoQeJPstuFQVJwrtvjFopGmPjSpxzjVXkSDxEacIfixmaGleMlOoXRPajNrZIXPDEfPJbqyIYTrTSrzuEqovscTbuBxYqOBXNvFKgXEWNAUTGBzjsOebIZGMMfwLyZpqCtysgXGOlBUDYKQYEnljEfTZPNbKUpelIzjLFkkGzAZVlrfoeWOqdWPSeoJhPCThYTRipfVZbyvAoZCRtJlPOxtZJhvMCpmEwCHskdCJYYuwagLTCoZSrAOtxUvnmpxUaYzARHsePbBbfVxeHOpEQeQxLahvxSQVLzIsaoZBtwnVvUPjDugnsQnVAVrFwhsKehyvfifKdoPSLhNsZtKxkuwndsgzlNAyJfXEUIXTBCutirCRfXiFXjPONVVuqTHDDdNzxHELssSovMoYMeCInssNZrvKKuUZMrYpZAMpFOoJZvkFNfvkPfFMArMKbXyhFHKUdEBIyDIdNHkfDSXNgZXKQrCTqhbpnWhdebsdWeBLNFIQeYKIWRkbIGvZSHAmcTPTXouSLaQYWvXCOOrDhOkxZASvNjDwrwmNwKrXxvtIUClAFNYezhSGRAiQctWSklMJrTjRJfvhgjkeSeNOgECOcaMnJLmQUOJqqiCNUkOtLsmtzllPcrWQkNIarSjOceVGktHwzyAmUukDLRDUcwjFVQJZiqhNTWmmZnmEwHeGnXCNkgzqnRWKPAjeyaZbaLHmqRljFtzXJENXQkfrgapJrtIdAFNbSEssGUmDHzfGAKATYHKvIWJjGyOlpTAXDrTHpFDoCfLYrIQSKlfbGXsRaCsEpQNnmyPFKadoFsddgxGfWhBYrQECAhkDbWaRLmeIOocbmIKEpfxUvgRGsMcpKFUxCynrxzDBdNPfCLIinvMHJcyIulXfDHFKtQkalfoCVQnDAWGUSCbovHAhkDHmghBqONBHnfdQGRViFbGYGTFHMsFOmKXVngjhOaosszIBtjJgCrEGggYROHtrhoCMqhGfVxpNRSjSbsGackewAMWqCEucRPYzMkuMLmXLcUfmxzfihOdpzqGxiHfZjYdfwrmYIKyoRnwbPWcBapDKYqpSmDcNRgHsMOfosrWgnVGGrtOSgXwXMXbrGnRhEylfreJNwRHqywJLEIVZCxyqTenThaXWYwEwNLRyrtVpBZhqJxdJIOCSPlsqgANNFrKojpDyIUQfGMSrsutYlRnyhxplADxOUmUANuBfZtpphkxgyAetpaLlMSUwtzkDwhwFERswUQOoPzpzYRzyuhqPvoLyWbmcxdymOSjxedwaddIChYwCNzdSTzlEueaFCuhRHcCqfNHFVEtrTdzLgnfepoGVUwzIPCBumqdcDMSTlDAjgGhPcCGlPOfZYmbXqRxlqgwIQDbfauLNrIKkkdGYShvMocjKuKITOPbYZrIcZJEefLOLtvKizBbeBOjYXjarbLuaUHLkjeHXpbxJGuquSSlPFZpcPPWwnKCXPfRdsKIOdgWjvOWcHvxsOvOtzzrBjfYmaAiBstfRkZscLwmqZhhHAooNXxKYWubWtGfyEFDmkZbeHWWNdMRqLWksNxfDKzWufpZqivFEuRMZkikTlmnpDuDNlJDHTjVLOugVPLuisRhYaxbtBmZgusldRxRWFiHghtgVrMyTYsqNcfhfuEKzbnZLlDGEAsKeeJXEhRIDtWUUbawrZkoGTdrcvlNzSOhvPjkcbQfgksautqhPdoWfBicXfvuKNMFCfNzXLiEgbNSXqhxzZWheYlUbUrmnBxHMKbcBhPjRuhdKFPggkLUGUJwUXOUrPIILhoefDjrYQzubqVdlkMQAlaiZWOORKvPLnxlmshQDIwOKoZJshuzXfIrcWcOltfWAwVhKJkbtjsCqlVxtVVcIwGlESRRMkpSoXbgDosHtYJfcFQCScguiimmIoeSJBkvfyxRcAnSSyInsmzhBuRzbzncFBXAfvJaaAxxNBGYRdoiCFTShdXSGwZlRdBcIZMCHzlWqIOzyrHJKHZBxDsdQGAmrmPjBCZGKhlNcDmSCSwRUQITMQbcgMfpCAvPPbSIfoQKhHAmOqkLbREeyOFcTrJcpeUbseOXzLSFlhXPUKLesDdyZWsKGLBpIwKuGwvfjESmGBzTZRhaoRtHObIgzvIVNVZMDGRBXrKVLFzCerXoEeBoMQzeghclrdbFKTCrXzShFyWiEEdgdHVzUwYBxiaiJKmhRPBtbyZcqEKPWgmEZqvtZVqzpoysHCTvSJtTjVMHOomeSZTtYJToqqMNyJpVIWWCGOnAtqTCGHQWHYLFENTREgbacgXyOthHHJtBPdqecXYWJkxRVZzFBleNUWsEFfyqggiTqHrfPmFLNOZgQeDJKIVbZEUkzYfGRezRgoRxSrKGYKopiuXFtzBvcMYXfkrmXgDYywftZiumccVKopLAHMfcCxaMNOIdUZWqIfiPsXlkJIZyrXdZZSWYqKrYjpxpmjWBpupHouXqmamMGSFVKZlNXxrNPDnTcBiISKExhqflANKtEXQpRmmaSpVZSDQzdkcpfQvYjftuvFNWgViKanJohLOSqirRtnJpmSkmpokdkebGmkkTtGflGgOHsshNelNIMeiVwwRJZvtfaAqGVCREOOIZgetAiTgBWrIdlbajUlEtcIKjrJSOvwyluTbXGyUuhtaSFMTqdYLKPdNvBjDKZXvoSApahaWsxZUuMOdxVkGsFTWdqVuSFOjUScJTMJEmewmHhmgCyDhniUGyEydEPekVvGOnjrkqRFeqqydXdbqXtmjlQfBesROOlyHJcAHtwEMJhLbNcGGjaswyeJnylNLxJFLjoHNqAuPMxazohvWAIKwZBgAFyxdJHYXMrUzFOIPZzXgGtHcrLXqUiWoYDjXIxkAfbNkeprCZJYgtCCZLUHYBkoNjnEUDZzLhEdXrYtjhwtpoPAhUrobZkhECASDFadONKKhfCwQysHQBVonGHPccsSCwmDRpNJeFWciAxwEPHZigWWtNNMqgWtwyUXBaOUwILUGjyrWsJgJMFhdUQoNHqYNHdVLItELyySETvLXQNJFHRWopRrelSkZSDVrMdPNANMnuxrqhHHGOcliiQATXohIWQjCIcdyMlWoeLscpPpFCSvTeJAFOZzxQZJsAMnGvMvufUSbLggURtVCkksHpMergBSzoJEXWvqiGigGRGdKlWjrLGsSvQOinmIbZnFtRuurhQKVMOuGybeswrCrwFQPieUtlYiQMfNgGShwyLppmLVGRniHstPqqzhEFsKYixlteVzbCkxEOdljVuSsJPDzemJnKdrgXmXdSYvUpEciEomqiYyfgTJQjomsrfhlCdyCDErROfqbVEwNaqCAuNSYoILpYMzrZOkfYvpGmBNAgDWLpXvxxchMimyHerDgUOQsqBKRwfTdTVHOPNRPoqVvywDMsCYAMfSOIDIpWGHvNuywQOwkfYRFlBbVKbkXGHfkPduftgPTiJVBcelbAVuTGZnFmpuIGdppvFNhsAAuZQDuqZlKTYtCxrGaYaabOHBCuysSpjSluAcXVixrgMYsmpBabqgfyVGlDQUnQQBuPJtUdUfefEafXExKCRfQPRGaCfDjiVnTPQmKdmeAmeYgTfrGKDFqTPVpiUMdZSkQQViLHYogUQVIstLjPjSsMwsrVcerdlWnVLKwavgASVWppBxSwcfZvAIevDqLQtLopUDLutCPiluvVVvcYWdvXbxApGSvLoCXRzlDEMzNYEQslkAtwwmSjxZQTtgmwXslBuEwTukrpqbzGwGQXAyDAcepGCWmIYLIUWmEerMJkMYbkKaKJClhaAcbehGZapnRZqsgUunojGnBNVmOVbxbxrcXAtMljSzmkEEeyTmNaySmmmcjNTavGbvXQeQmjCRDdwTGepPKvAiyXfCBkmsVhgjDSoUStknRjkWrluRNQUUTGAGPESLaDbSMHMoLITlnGUOdtKDCSCYSNVGfaWAyesYwReEiQtnbOdtexwViBjMtpvLBYlXMxXFfDqtTQEoOtUJQdfMyBkkcUzSPfuAfbeiXmyNBQMXmpqoyZFxvmAyUyRleVfJGzGBKfWvAaBPYWgCIIudSYFTYuFMIsGtDGXKlzoPlOqFeAsxpqvoTUTatVzobPJeYTPFjpRsFrcREqqpbfmVAKwqKoAmXnnpoFQyszUqdjEbMDSYkHZncYtJFHWNnuvdlglAmGrefmdlEShOJUUpJkjbXpjdoASDYcIHpBnoSRUHIUQIqhaEtxuETioAxqwtEuvCwqFzHkebaHSDKnAWiJsOlzvMGBLUyPDCxZGGRocFmUBxfAcWkMDIbFirAHXvjmClVfcUjdgiygdHanhvaEvNwrjJShaafFKaDIaGubovEdcnHhErTQEklqzSGFQIEcHWxCwUBJoBUErlCJNapchYWoPYZyaaoEyJbEsPYxtLcFTEzvMkqaWNnwtAcQGXMRZmPAXzINqxGAqrnlCbyoFSaakYlFTQaDtiRNXbAAdzbdsQEAzySfdBvhRBJnIcDUSfHKHeunQMEvFhEHLbXVhhDdJoLWZVCqMzysBycXcHsxrYGAqRLPfvgBzMQERvNLTLNYvfHtdbcQMnEjcylrYpABhCXjlaAzaWwOFLabbOdQBgtbqnNqBPbCBLcOshMdFYqdmIWKjqkrmBizYXdAIQxbqAZXNYmuEbpwFfYGbvKqJHNUmkIWkmDmqavjFZKUdTjbpkxyvuaXCCJURtZxyEBtkbukwezojdPMGNRpvBNirFkezcIWqxHhKWcpQiwpzGVWJWCLQMcPWxTcmWXIsvHVDcxvsNKJzBrPyawCylgIomaEKiwPdbDXDltRYqrfvfBAiiQMOiYjMKghovQEcoVChvZqRLwOSeaLiOTkzOhmpHlXTbrxaZUARBXHCmIPnvPGRhqXzMyYOXCdBibRXkgigTgIkTKGugYrMfRnXUSNImfKaSZmwoeTLkwnOOzxhLlImyJEHrZUuZNCBbDVzewBVOXAGZJYjINpfMvzwzqduCmZjIfKPkdcKvfJiDFbpUpDysfcymbOIeSpfvenUoVFWFFTYnuyQDQWoQirlmhSDRQYzKaYAxNjycwzJBpXycUhemhzggmUqZeKwlQTzgKFcmnGkHKMBzLXNJBpBrmsIenMWHMhsLrdMhiZojUqGaRuCgruWTYhrwmiUexkHAxXSKNIqdfSQHHeCUmuKASOZHBSMvpZGbRVZLfQpXoxGguSezVxORDMZGOjWRWtuPEYpaakITEYQRItzvnIDMferppUuhldKvARsfXAUjOlPXVgiVuudGtGwMlDcHEZKQYTXQTzjRsuAUvUnoINVQwQHxIdZpgEeyBARZzfCswzhBKWXhgyiIAwwaLbaeVyaavfSWAPSHtrZcwKojrQddaWUeKbHfiVoOPQCgPybbcyotYqXbYIiUdzDKaxVyrWBTnqNXlxkLuSBakzVszWcYmjMrBHxvihjbJxcqSLigwhMiNSaUfNrdpMxbTjpbCOnpzxDevTjuIUSSlaKqNcTiJflkxMgiUblwxhVzkofyDmwHlGvUZKSjofychOWASUDHhVqPGfriBslpIzqEvLNaJcPyUcHqnelNijAfgdRDYwqIUWhwNbsPVvFoEhOefrstoilShzTfBaoaqWULmsdzLJqhcaFfPzAuohXVZBeHGTYeflOPtVcXfBpYuLNTZiGLXGTWJFsGuLisMmkOGVjVYkldPLJGjAmNedHSuDhjHIRYhQXrxrpFRmMrZXynvflXzBTBuRxroTwwASmzROSQITeoqtSfKZMydixqDOZFShJOBGceHbSfMmhfweRCvMJGZSoIXOqJfysASKnDTjhFlwXPaksCGSMEMMNrdzVRABzMRusjkfchTAoCNpZPNNpvJbhuvTOQjWmOwxEmdAZhnoQeOrfWuzwWEusKwKrVaDckUEfogcvCggGnFrwMOZhdaDrCzhMCOVmfQiOTkaBrxDsWufWTIFQNudjlbjhLfYpRbbwpOPFQvtYLyNeaMHPjruloUqKszZRYKAdczlhUviGLZukGDPtVfJpxIoBusUeHojgvTSFfLpQpyDMekrQStbbfbNVzYpBylmFiWwmpHcOSZJLOAzevouQselSmRwDZXzyLXmfpfyoEAUWWsEDBsIFPWbkIzKjJRPMnXYXfkNjeOXHwNPNKnOyOtExkEzJYoRFKmNZnAXlUWjRIsoGbIxfySlHWMAtQGEGlHDAndWLSkRDMHewnwqrYDTJlefzXwEnFzBZgZDSitDJeGxzLYxUJnsvDCPeBuQZBKVBFbMMJaGNHjvXvhMzxKklHleqhydQeqvypcGToFnbmDTcfisHDOUZXkuODkcPBLXowabZuemfkLtNsKRPGnoGaGqlRyAuMTuoWfLMcwGtYUeukdSeabXcHQFpWdlqJytJXJgNUYPqzgvcHgmDZjqWwMHthrmUcGAozqXxkULORMzNSgqqbJuuFpmpxczRxLRPGuvXvAoJMxrikwHPPUkfPULKLnTvduzMGNtvEQdgKssYNnopsfpejDvIWvLqzLsSIiebHtBiWuHLDlNpLBdNVhiQenRTPXMjXTTuyGlIEJSczRRkkXmOAjMIYBUZLTEYxBBKGXWPpHwHmqIHWVhyaaxDxGxEREzPEnGdMWCuPYINwXGygDZuJjJYZXDYnGynkMZYmSFFCGbjVtOIcfrcCVTBKnPzSwsOzXOxqsSxOKkEtwZBcBqIpBOwutsuWxZPTMTdBPgqfZJYHvkYzjwigMjPeBZrpoTCZjhlFHtfmCDPDUeUVRduYvDiSPdCrofEcTmxRwLkGMQTUOYJSBbNWGQVFBxwCamokbXORVzOXiHXPsfUiKmxSIaujNwEFaoOJJugVZliZGUdABQjiLYRJzGUQTduMUPJXpEHNwCPoIIsKojNBTHICgYMRjnjZDBFlXxHLUhlJAqlftXkbYxOeUdLEOkJtNmjUHXMxCZysraVkntbZliDKyyGfkqXVhCUPwGkzvrRqWWBCRWZEGQEWooinPbFGjScChOlUEGfOxLuQMBoOfitYjEfvCaFuJCeErjoqVTdCDaWahEKdYXeLXAtgSzVYrNCXFnWHcbHbVJJhsbTuwCLqDUXqgyImIZgIvHttNlArOmTnjhFNYtuOnYFXlUHbSkqfLeIUtznzkVIJZtLaufctqGkzdPlqfVPBEHgnxaEWnEuoDIHepWcxlqGMpRTjzwCqdyrruwtFCdrVAqeaZOvYZYtSkkJzsirkiFlvgWbVawOusCPdnVvvZRJqaXJORRNuzRfwMcyHhyMElBLZfaahIWffrjidcTiGcWFMjIkdHRjUJZmjrZIPUirePzJtfEGVgDOJPqtEKUErBomKBaBQtxntTGCoQDVVLgQRforEUFkRHpQgDgIoGMrsiOXuStJMigUzCvGNUONYrrmFiKyhoJbYPpDYddfpFcYMTXmpQvvCuzFkHISKhNuUFBDrvcXeuXmPNvLeLxsVmuARuCIWFLyvbfnUQdtSXlECjQiEpVlmBOpZosbffDDjTffZSCTtgwGxnsguFPTZuvBRnoMNkyaEMJyEddANTqJNzMHSIeOUxhdbibzfBUDRSELxlvznriDUzBisfdSytAvrboydEmOFMAeIYsQLUIvqzcWkZziFsXoDOdbxkziKsLOgVTQfWkoXnMWDRMJbMTCocVZVeNqArEGHDCbHwjROHRwcshCKGVUFZvoBcYnWwXpSZKHCcvqKKtBsdlYTdFJZfYdsKmhUqCGSoiqBFxSmjdXXoeSOyhJODhnHBboIAjFRYJjKZAxBVSVrTvTDQpbfZZljBszqrpbJSHJSMRKZvAVhPeSczyjAVlIMEiKXVnFqXQzBhqQNFMwHecdJmiKtWOhXDmahVYVwjUtMURvNbvdkFRTBcbMTvbpqLyYbZUqxeBcdDVUMSwuEtGDXyBnVFYgCJbmfeARHeNkghPILynrIAWWiGqVCncNxCQqvyPaQXPtecwZOKXcppDIHXxCPkrAzubAMbobQtpMneNjwrNfbrdQstWRzRJyAABkvcmDaBWbqbkREqjZFfojCqIvPvxqnMVYBVyAccJEljapZYoYiRNbSQQTwuVIyGRerffRTRAXhVmhGDAbaHqTuTyEfWAGaqrsPyOEkhNVYtKkXodhpzYQtVqnPLgyjVPcwGRDSQwgWsLlRenaKlZOARpQdBkIcyezIQEYtRSRDkWgousfKiPzVXqxRiOVnhRArNSoBtYlAzYmQvObljoSWxdAVuXnTJLHjMLrzrZTxGDGQjSTuKyuUwmgraPQSuNqMthPzxinCXcORPrxPokqJLfhFnOdWlboXfymrpBnATRRlJQlIJGMShLNEIyXvoCFlosHcbPMiemJgrmmXXTcBLgJgsmDlnUyBmdnbyXkzNDDTmdmUrEYcsBGnxbhNbSvTqnHhgHpDDPQQkzpsPStKowWMlSnnacOpWVUDeCwUaolgleFxbCpjBiZoJyFUySWCcnofldBAELjLGxTRqWGBZrKcQXcMKDXyApgOHbyfxmTcAkrpUAFLWNSryMQrkuSOYhdKnqqjXlyOpcLxRzDBcAEiuphSjDXZylAlLOSuZJxvCMuBewpAvHxKMVhRBQVonvfuHnlUqQALyXxsnLvrXMYjdozaWAmCQGVViuKtxlvYAeLxLnkXrbavluICnmYQcAlTOfCIdLWWPEVSSXTRMevpApunrkrwauXGOrTJfOJiLJHBIOGncVqskGQCSrmLgLnHZPUfQiJEcKfpBJLXZHUWidFlCSnsJJLpILtWsvIDbahVpRxowZbanecHPIPyKxXcqaYPZBPLkNlsUBNFKpKoaJQNaeftqcLOSPzzOMYUbWXuVqLjKtHtqKWGHWnEfJoCiomLPRNJpvZHmFOWncgXmiikZNAiWLozDAUXbdaCRzqPkxbCuOpMHNDesuebbpSsOREEYCYDYughEMVzYGcATnEeIiZcdfKlwgohkPSWgnFSeJFqIuaQvcKWqmTakQRtmvFEfCMAGNBYXwTKFudBXcHaNgvFGOnNaNHfZaowmkIQqOIGWnkFeOoBgCjLjdAPiDKhBICnzejEbwvWVNEdVnnlsiDUrVXLjDaqBNiMxypvMaLiawTZTSCEaPQPwnIIpsIxYzWOQjUqMLAqBjkdUqlSlKctUUhaxowMVTsnIddaSxQWsRMboRYfvWjGmPNINKKEzsUQPdCctyDuZssNLAaxZXqywtwvIifbYLILbHjkiogcMxErbqACzuHIXQUyGUqKAaNDsufzvBJOnnTSkHkIvniUmCWJFuGZVfZNRhduciKjxrYOBveMEDWWQckmKrqYsyOjJKFUGChLwUjAlDCxpVVHRBKJnMlgOjIhRCFXHpyYZlozHnXSaLpusFeLlOjWmbTdTDuSPzxcdgavbrsjJlRWNEKqEoYtJzUAkOoRiAYjWQGkPkvlpirphmrUFbObUjkzhwzVMcPfULijtTQIEYtTkXtnBLIDdmaKRCcaIFOQjMiHbmefZseOxyUYtxmvibimdRhVogBoIYeRVwdHWdeZxcZFEdJmCTvdKNYVQrdTxaXceOwbqkWnPVuXehbidHglCyRPHpjKZxNwvxeuveCApXROKVKztMefhdsLowEBEMtzCbhJFKfPYSwBFlyDfEepdFdjkuUrbJkmRhxFriWBiaxtWNPIUNcVPDzQbbzXQwNSxKpUHOAaNgfserLeOqayywNIDtZtvUJWFKfugIPzyzlrisXxGXZsFsjUVLJBQPorJFbGNbFWEoAjIsEoEOBDAUWunrOoUVKwTwzsvNCJDUYsPvmDXLdIQcfqSWrEDYvczGRAbJyVBpatrBQHNbFEbRUxEAjKjgefLHCdQEVdIUGbyPnDLqKmpReHhUGMxjWFUUPysAdThAEseVKgZjNcEyuBedLZkVEBeFUkaYKOnhlSsAABpsYJkzxddTFaQQMDJsUHqPcsFAQFpllzxIQgMQKPpzWvEdKtxPLqgzkNbtpPbQnwaEfQKlLqfAcugixNJMPLAXmsMmopsOQaTnYsFKOVTEHeuvKICfUDMryuNLrjrudFoMnpjjnLakFRxMojBBGAQjbDxAJSUmPEvGaBvyqguvfCjzqGDxVyBhmmEZrjKwxgcNQamBjowBlwLmKXYQRDdJtSfQYdMDjeYbyuVCzLumNifJBABtzpoXUCgjxRrOjXrhhoskAkmibxztCiArOKzbraBhMHrUAHqvRwIECIfhBZjfWfAaizgurPshEoFreszolcqaUzmPWHQMxBeyAotEebZMFWMTKiiJUSObNezAOgxfxDocBpcAUCxkKgNkadYMBWwJIsFivbeGwyBGjxXgidNIaRPOiVOLSngQyBgAlvVMmAMUgYCLcraXORMZSINXzapwfGrgNRGyKpPcJQkSNBLyNqndlhenYkPDNIbPfnaDPBxJZwtPGBGzpVdbKRCyrxKIgHGGQejOZOOAKfEzYcIDdIzHUvVNMtPwrXFdgADSYmKlzNjkNKVHitYMqrxffpQbkpQXTmkbGUlsdxizNpDNxzAbWmeZyMXrZCyCHdAUTKnHvZkZINaHsNTeMFMNylEisKcYsDNTkmxtqNjtpqjFLJEwSAfqAmZCwKceQbxhPfQWarxNMLjCJSjqCjZDqBsQbPuLPvwpmBQgkLpBnwghrChASIGFGPJAJeqcszVJWMlByafSSyxSLkcDiAPpsPKyGYxoKYAxWcZngFIjNZxoJhtEJyZnhLqCwlbaNwVfWHPbSLqOrLFwUPowOluQwqqfbeWjWPzTXJBlfaQBoKmeIodLvPQXsAPcbyWSfqCmCndVdwQkQfhqkmZdEtZzbBqpVIrpaqYkOcZIsiqaJlxuRCxkJkVKMDFMvsVkTousnQAlzQWhfOJeNUDjxCmfTNVVNBiipsuWxtFBMGJNxaoNOnhrgWAiUkKfJiQUXcapBvtPlenWOsPFdasTVrTeeybUkBJWsNwNukRSmeSNllLverUTUWiBZnVQivxUKgILkHXMIJlcBPifsSKnXzoCPBEBrXXtdhioiAPNSJuzYBZvSNAnmyHFveDaJjPEAEChBTQGfLrcgzPgLZVBrxzSCfRwNpdkVPqZTzfgAZuAWLAdAfjhYTSKIEOYbgRrxjcgJVkPqiqcovxhFIjIkQDHJPqDTRdDrmKfuiDtaXcTnpvPpYKAiUBWpqnxDGzDWALdxruzhogIAurULFTKQbSRFpEPkuWXvMsBPNxKWicpYXkwNxRSkwSJpLuMxVgEdQKIWBDmixWSaaRBizgZggKrTQdKAeegesEehwpNYgtopyPuhroJLuTLogTTNBbMaHUWHWznBNJGmdADxIDSIphSmPVttOUHuzQRowVasylihlFHBbkBhtPRHndbfjiZVWuZKMTUyKPKoMlpllouikDVMyNMyeGdyXEotWYsrKJHLOeyPUpVOtmWyXjKbMQnpEcJOedmTAPgYcaEOZGwLoGiIzDcbiIwksDLXKowpLdQChqQdqfrtMrbXDhXSwBfDRmnfpWmmmcZYVBEDKTDACjnPjsADAhnqpVrCurQvJjsZBnUxBPllBmrTbUrSoyjrlQVNKPDcrdUyuEWnFNnetGegkVbkNxUDrmeHuRTWZCvUVJpgZBrKvUTEALWXOZXJGFRcaQxRObUfJVvzQVCFGFDpLZGjAlxZBOpdTMFaHheIcYGhHBablSxeNnikiLFCZHWuayyuaxoTxDRbHAtPhODPhgaIvjLZBFTFzKRPyANniLPpeEnzdavLjHUbYTGMCDvJxShNjRlvusmWkwQTYOXAvXPXSGSwnKWCZJvywASYVWzbiXkiNACzriRqxhmpdkKfQAMJHHInpItZGmruyBRVqeFYIakFMLLWhNTYFGFzGGVMYhKNZLSPJOmuLDyjepwTjygSbvrNvhQLiVkIILxYZAVyGzFKOvMBpcqUxyOsrMfczfuzwnmyOUodKvbuhcuNwJEpIktJQJPPLQxujqIyIgtPSRtmBHyIpKoDpUBXIKDpYEkFVDkeFOKkxFCCrHtgXxfFeaiWazfQUsXeapyHqaWNKCULDoQMngPZJGzvEGKLmzIKZwSSjbrmfeItqpBuvnfRHZgPwxEAoRNJtwfqWMAnghnTVwCrPbylDhSNbuBsZicGONcqyRHkaiJAsIgLGgLNAibaUEumsJhUQcCopNkJQUSOvabyZQIorkmkYNGAObPbsLxEeJqFNegrNZNcmUylmqbASkVBOGLyBkpHfREsvTwOXULDvzdSNjqoqXtaFCkstvzEtHjLlVvDeiiEMIoLcUJBtDPCQuZdohSSzFfGvRyxHpNFbRCnQzOiajIBSZIdvZdoJLKXuRnTrOplAtGXdpLqkujYtRXYVCaLaxkqOPEKIsmxjJIMIzTgqjuWKOGybsTOPsyrkewYVDmUMzptsEhUOawUrzNbcVPPWlhnuRMyxDoOXSzylLOjouygMIAMudlWGfuxCvugUEDgllAJttzaxIDmfBdRncBlDXUGDGXGBZxnZobgdJXvZJGfcTylHUjVyNSOQNixRHFzHOCaiNNynAkMuBgQdAuLfxaXlMjLbIZJvLXZhrDLcZsSfMHHMgejqvZpSaGWFnfDGsQMZIzYxCOvnJgZksnuFUJCYizuqFHZxcRKqXlJgGOmCdqvZOGQHfqzCtVBOexSpmMQBSSBSfhBSgyxeqEuBhNETWfgzdpszuUzgFbnfdzMKJsOtYZDlcikxkkEHWwdLzFsGDtsopWViDHZFkyHzjMjBogbAlbWDLVCQKkRCDQmNkvzWfgaTiBmViUnnqbBDeQAYppaCtgroTohcgiajxsxMPwoNDlErslPYtVIsNAxxXjzfBLYRjGdalFfBBfCgPrpwTcfgVzuHZPWtuAfVuzKlaGtNVedKxSMPndsvUajONRpqtZGnwOZhLRZykKhatcacFMtZNhAqGQWzegujcHDtVpwAbrweTuOAsrVJOhbuHHnLbrHxrZuVnLGBLmzWEwjHRswZQTOzozmQFVYjnmWmzDfAcBiWmxiurPobtvzXwydOKsaBNWUqkVLLrWuvFsSMGcQFSxnvQFXNFqLkCoRIhxcTZAVnCLzkQnuKTtRNEZwAlDRCJMTcbaeVbEXOaUsGNvVexlMzsFoXAaHHLhcuOLvXnSnvKaabjhpcCKMvfTMviLcRLGwSHCibWAgOIqnTPFtRftqumQPrUWmRnqTwkIvnbmzpEFEEAaXYGDmXcetakYMgcFPjDGeLnOXILlhtuVwaumWARMjTlMaFFVpqdmklKCSiUIbHeJJEHAfxYnPeboIaDPIwEoPjEXkVTQJqaIgQlKhpyAnhkxUZYuUTOVirTLqDofYlnHoVZNoalOtgasrpXnmyNlMZpJfzDGOGqydjJADTAkDueyWJgqhWXDsNEBdDnCTgKMqsUuzeKHdkVQWKoFezTIkTEdxkUZJyzVPgJgSstreCsmjqatMeXgDdKiRbFzSHUSvrvXzdtEefRSkgiLlTAEYEThNXPdNwDPAHSSkLhSMjDMPuQNOveXvYVWRaBoznmvuBCZhdsdVIjsGGERgmOIanwbTWkLMKBpjmIkbjOlOpRVQElxdIoePVfJlodtYZBQMXwEpgKvgdXvzusNpJvmqGALSwnMQtlWZRlmkFVpfPWphWmyLEeEFUwvdMQTjSiZzsuxFLHAFKshWaIVxyXaGaOarbcWKnXOzAtcPkftaAohkgAomsGrJUlQLdgKYgfXVdqiyrxYqgpHYmonZAgddlerfycYeJUDSfUpojKvOeVHqbESmXPPMxCpTQZtpercxxJsjqVLQFZfxCDnxALyIJtRXHYftJUEJlnPHUaGRSivUDnAThrzSEANJFsGcgXpOouvyzIWfhzkUbVaeRnHCmdmkShTGxErQjuyJfljSBGVjOQcrRezCuXywZDWqWTzXsABtruZJScRYTQxsRERwptCYQYYiCtpxILecVUztZheJOaNPVjaCoCsQfIfQxlcBkEpMLmpZqdaJTljWGGCFnSXpzFXsPeoFUNZybeKBjDJaqrhGDbDEHbtFLnqYRJczcXBaeCCkwEYUMAWtlSoJrYFnZhVnLWWmoGxQrujuLbKOZdNwxNheCCvGHdEoxvvKYWIYCoRNyAwgtiONAweNCyeOJeRDhxyzabhKbJEYGgLvLTegVsVqLyiMcIEPkbicOXjbgFzlRhYroZVrblVPslXgKeaQFiUWTVRKAPMnHxvhWnAHQhJmGdSiXXewzZjtsQMNYFyKlRqbnhqJyEohbMBdorKvofJKeZZGoElSqyQObxIBAHmKKFRtnzbZoBXTorrfcxWsMONQgttWnEuctHHCwrQwYkpkmEEGMXasrKTEMNqAJFxrJeQlqHUtqBFFPsqbTvoVOqioAhCDRpKZgvoabESclAgLygzQVCOgvzxfwjZoELVpddJIUIHfhVyOrdvidNwpRUcbeuulqwzEshiiPLSwvynUGieKzmfDrwRodcbsQBfgwNMLoVZJBgDPTSfVhBAusqDDrfDhxsmQOdUhHPKdxjIygyPlRIRdQqCUCtoFVEMuVaDBqiMiRqqHwaCorxQUceqXsKRYVGVkGNjXReXZCNSJLPHNmRLPQrqKNQvmncdKepFVcMizutGewoUwMnVdyBkFVVLGLVJgUuGNfcLFXZHyUPPcHoidBGkMZHyHzFnUPYcqCdwdltxVXRqrTtxjXKwXBZOILSyfEwWdQJKGvTNfJvemgfGjkrqbkUvvkbANeOtFBDBvfOIYUTRhMfVfuYSiYwRAGSJGNIwBxUfpDhnneIiwGjVKLDFXYGIzzaBejyT</t>
-  </si>
-  <si>
-    <t>miALtdmtHHAlAqXreSDDpZJVHxLWwXeFDMcdHvQkikNaHDIFvCaRjCbglyGdsWbosxNqiYTNFEgBQeohxjEnXhHBTXhuHOPrRNLYqSXBjfgiObEyPrAeHeDFTBGMYbUZTBOdtuNZVXQmriOWkjPmsoqwzClovdYkcmQJEAbvqlQyzvcDzNLHuYNyagfJsigqIqgxWMaLeJlaXLxoemyikaLSMlIEVAHFYyNZToySpJpTlcUfAQRoWzyAMpwiNbPhOKoWxKIECQCSJDnARFUmWabxDpMDERuSdupvzpGGwWsaryAFMGylEVGQNAjPDuumlpfSnSZcAZElMamLTCzKQcZPOAayGqaIhNmExNaiMgMybdAmYsqldQWdpbjSnWLHdryFOVCLvqiaLTcjiRFRmDKbAUpTCWZxhzxdHvXAZTzDZMlAyFGnWhdDgrdTOdbdabLITjBLlpjoxZMxXPvssibJKLPBUMUNHbVjNZcHphkRapoGbHqrrtdJDPZSTMbMHlTSdCKFhdOuBmTnykGfTRlxdmdvWBCEzBsdSpgEawCEthZXFvtWTnKZOiorttroRTadKaUlwOYvjBdqLnKckvVybBdlyutDChPcgmSJrdbLgqSptJgbEyqyKrBEuWRyqSHWZvAbyofvrirWlNrHxAHdvydyykPhSKRnRbvgDEXXbHgfNCGZxAGaulnQwnKtIfkdeYEcXGQjiesgSJHMteXhshfltaBjbSRqWJKSTeghYnAAbBFKDHEKRIzmAwDzlyJLXAlWMuWkQTdluoBohfJDCkUwKelYXLIsQkWBwTJQZFyaOERQWURwXxfvdfvkkOwXaYdEKYkJzGdsEoWuXGrxAHOsHsxAeMSBtbjUaADdkMQgujVOgUxHgqMWACHkdJoCZRtDkAFFKvweDjXQayrRFyQWEuWNQfSqCwgmRCMVwADnKbGPxsGOtvpoBFEbedqyeZNkpgFrgWePIWLaIwOszHqdLEdQGoIfQDUrHKvCbiCbGuBVlORKosmwvssAPFCyntYOAvJTnbzqrfFNSSXAKzlqWTdNFSPwojJBYbmXmFxKcDgElXBkmpLvGoXaVZRJnQDEWoAIoQzFlvqWJvYTOBayhhsglbPRcqOGVRbDSxoXzIQxishzldqbopYsHZWRVIoJrOQQWOsYpRaOQRpouAHPJkNCtzCDZZBVdBtUewlkagqekpPNIurLKXiKLeWyjsyrowEoVWVRYepJzrtLRZLySgSYyVwyHhkrQHCZhGzmkBrrVVragYzRfmBhFinvNWXPbUvBxwttYIUCWfWTFHhGjnVYUBfpuykdyMYXFJszRLmMXlPQZjPGqsztIkJABIgztUnHLJJiROnVgJBUupKKVDLyjyFWWRFkyuJmoejRcvICwUjHRaSCytphMUMJFWunwQcmoPIpwLGECVIpoxegyHKdxwVlAgZLFIryGTgbObMCjmQUviDUGhrDcKqNQIQqGpDrcZJcElpoOeTRFeTApwvykJqOISFTwlhbLSolHZxzdMLOTPPDlllPttrstdDnnZzytTPGvXhmhxrCPVeerGAqllNpEYfeBJgxMoldndOrcCbTXeVsQkzJmjgpYXEjvHErdUpPICPuDHwmXPkJuVBJMQBxvARqnsnOzOTTJYpMJIWaJwQRlBUeUvIsCzlkBmWUFEErPrcGLzZfRIXfPUjyVJmeTJLYDfLTDIYpNqJYHMFEiYbOYUueePDTekBQkGiVTCTGGRUBdOMiQLtLeRiagHSRQxcLIpYatOWtKMSaxwFBkqtJcRTiDVqInkpRRwPEueTUVWszJDhnMJyjpWswQJxadhYGCSrBNVZacYsKTvPxpTQIVwjXuFyPHAJyXYJehxjlFQxAJiGKsrzBqqWUgiYTSywOpCTJyXkhfWBpBqxpANWwdxRHcDyWHPMLKpbJWaXWnpJouPNAeSAPadzInXPowvTuojzEboQyVdiQLDYRXHfDYcmsbMLpMidTJSlXVcvTdNVwXDhFPnzxkAfAhkwHxLhsDLFWtCFOWQgeWZHWSTjJYqrtNLFpPeRawHhTSOfreJPkGejKloOdybOkQsupINOWjCpYEQXRlOzqOPSlvsRHndiGcryKEboWCHLdNczonojpTVegbaSbebqFaVoqucrLjDAHPpFUFYuCYFXSpjpzrmdqInfRifenuHBTdlCLDnZxqOfvDQFcybvSTOFiQCYSVFEmQimDvHYSBYtFdEWjdlSjRZIbfqHcaxnqZrOFPuHwfvgTJziKXummMCBLrSxVHaudVAoFVlIXGHgiqMrrkTAKgPHqBfTpJpEpbKphlqaMnVSCSpAcrnIxFSDoCCUgxXThFAjuziBHhhqdIjnyYKbwBhDUjnWcrBCngFNMSGANCZQCNLinFieVMpIZgcatEoMcHmJiWnNAuGohsEjXPaEqJXhKCeUwmuBgATHMRxIanZWPDyxflZJsHuNoKOBvFeusKabnyEsOQpItuCsKgDWvZIQyHAEIXJvKPbaDQnTYjvzqOejngEZVzhCjMuWMqpEBAUGVRILKWmzvhcQeEOAOXBPgTDoeeRPONqexckhACpSmrgDsbdunLDMDkCNJrqtfobCdAoKsbmaLyYpaBwyznKzrkOfagleAtUFEwrrgEIXVViZoeMSnVkSNOrYEYVVrdcPPeHkzlpOfiOdYovcdHamwakIAQUTRQzVErCQmauYSPBfzsbouAMQbtmNvXGLQsqTYScfEbQlcCKqvSAZVDeUPJrkQgNwgcEkoNgWpJXXhVejcltswYCMZoaVGsbRbjpbQnzfvXPtUjtVUVLkjfjTReoiFuCTsBlSBgdkCyiTTvGNVtQiZWuPuOPPhSZdxbaLBEYyovtcdLdcrPHkpwJGrXhdLSJAhqGvjOWpHXblkYVCvjDVkGQeZnalFHitbsNKutrXpUqxYaHuKAhIrReiLtNTQGhtEARLbQCHUntxuvrufAzrIfzHBGlGYkfcQFKxTtDLcbbGKwXremLUpkgQEKtERWfgHapXJHRmlIwAHqyPjdlwKZYeLQkgbqskBDXxaMgZqJDGWyaksehZXajgHhDphfTyXULWQRcGwTnWvfyGTaHUYaAwUtNelaNKhKMoDeTmFkAXrISsMhHrSzQyerPwyFQVVILUlbJjJotBTofbFwhoxjOyyYntNDrJbjlqPIkuxsrJyBdkSXJHnIghbMonfRmKAOJbyVfgGmNoSuLShkkKTAIXBGREHNNAhseheMonqOmiXsLcIJoYkBbEiyBoVYbQYSvyNJxstXYabbXNdwZdgNpcHVxvxXafNwKQyJSZFSkNfHShFqEUlsxrHbhhmqgzkTNVfqKJuMTiNtpVlHFelNDhcGoIrkfzoUuPmLCuKwLrKcbtsnJLXNlXTbzxGqoNHYmHtAxGtZIZzgaUdPMEOclmkxCGPLxYftKZekTCCtkVlhSbctjyijQmDxUOzfdklcLLmMfHhDrNUpiLHmQrzXxsySFdbFyIoxeEHJXpVPLAkfdiEfihWaOvJmtBxddjyiolvNishwcESJlReApjhaHdWLGSqhqBnZWxTVqcVvOBFMFLbCnspQyHjTXHrKvLGxKBgAcrrTZrJuZWtcbIkSHzxpRcqLgvJznHBgmCZgfzuHQbNdTADpTeQcLAiwTMABCfwgMDjsQILhhkpFNkUiFoqfbtyTAhBArxyIIGFTEsHNlYqZeXWAKFsqPsllavgVFoYLbePxEBcrVfvUMtasysFHtvFHKIyJyGHlPBzDkIOZbiwDqLNqPyBmjypXNgWxygAIZaueCjKJXKTpsdetNWwCJCrZZRfBWYNzVreWpFLkwpyZJjemciZSQyTyApeWYCIqpgiqIUIkilKyTcHoDiQSumrzrUdFPzjtqnlGVpILitOwUAvfLSDLlKmnCMJDbKQsEPNcvLJLvtzyVNTOdUXVQqdnWzCsqGAiEWQJUjGLBnipQXuSzalhOKeofcrbQssrgyTWfAzWlVCGPVEipnlimyQMjbJHhjnahNwHCLaGWVRLycFMiSjBsFFBNgWjuaKVvFoICPOQAOoiNNHUDOvInfZHysLZPSBLjsqJYJkTeDEejPHgFYjwkKUfEYoNrmcWnKdExkbpIefrQyBgCSSLzoEdwJbiPhwLILEQyZRSQzYVbVZHBviKRPrvGrOEPEZrdCKDYusGDbkXyFpnijKdyUjOMxFMuNbsktAkJJpKlKyWYXJWGmVvyUwSNmbNNWoYMYQGCfimoWXbQoJVAsWPkPsLFLVQVePxYLrrsvSBVvIZUQtrJaYcEZbuypiAjznTUANQKeVmAwXKUwmIpDfdiamgtpYenTtNAwpoLbnkYQmaIwvyhEgxHhegOflYKACkowAeyVPPKeJvtIImtZlZIgVYTmVYdMRjTuJxAuJDJTFuxvZJapkMIehpHqmxrTMXIsHkcpNIUoenZHTbqSxUWPbNNvbRANqBUpvyVjwlVLIVeXxoGKErerorycSErVoaVxAMQCNNQPeqEcXWAiBEMqwDDbSgncMlnlIEqfnGMxxPLIzOtbaBgbSzBuZdllpVmAlYcHZtudRLAuxsVawOpHaSTPRqhpDyTYVQHQiwHBltDszFNoMDgsNLvnAFmmTPeRSQDEJcbuvCMOGMbUeUIAkfgcgwEcXyJCnFgtrtgWxOCRjUaxrmsqwiXspJeWTHZURbnALtSzqNHfVQpDSalSNaVCWmiEaznOBiZlceCqPEGaEudXxBKaLBGRNBtMoTHvLVvvghxLxJoBTYJgYdWaYuxsxMsvRKpgWGDNofipKsfwWafJIlayUytPpcrVwFHYhiorwfCyGsbCxPFNWpFNcXwVVkDkHeNcdLuKgCsAtugmearzKyuxvBzrtdNwTDDQdHivkBuCdbExymoUefprgzFaaQdXfxEexIQLcJyMIhlwfKnJMrINvhqXRwjcNZdxCLRMdhboPGBVGkLIhASbrcNpNasUBymNdhcNhagbxzoqsjRsEqoHRSLvDtaTWEjYahFTtIRMfurVeJgetvAFIxmJlyOEgjcTFiRrkQBeMsWxlURTbdioIEtQJBTNwgCXPDKSENTANSsqAIxyWcedHMLGKxocjTeYpKrLQNJrXSjfLtvWQzOGRYPqJMPnexHqhFtXHuQAHCeLEzMjmoJOHYCljDBACVpNvRfTGCoVSOGrFyJbkqsLbOlEWAdChQSydEDZjgLsocLLerTURtjhDejVoviJuMVSYlPJSUApYIHggbrTZoKmdHTplJgZkJmffXvTOodMSpKVkqpoerIKrAphRHVbjTfNHEwPuqLywLkUbCOKboQlbRHDDwrWVYDpvHzioMlErCTnBFysGsUlMggDQrxmoJoecetuZbruUpJYhAPPXVHdJUEbsoqHJJCRqyiliFWSsHrXReKBICQypZscHkEXwuDbMQZqSNbNCJsRxNnpzQEqBrpQIuemfoxojgjKjyaxeDqKbJiKasBJVbGFvLPSeAGqgSqJkAXclMUdckcBnEkPuXttxIMagjsWvwHcLLYsVsAvcmMhaQxKmlMTlnPnGGWcPsaNWPScucJvNaPvhAlqWyzWZlKdXdkIDRaEjnQjyAzDmIFntkzTSCgivhhRVXKCzcBsFtTMVEkEZPztSSGCcHpRqEoPWmKtwYAelwrDzKGfWiLIRHIugdLVlbbnnMFTRXNDjDydplEJLZdMRMAgqPaXDapWJOwKgqSyciSnRbbWKXKzLwPSgbRpyrVgxyrLgFiypGpESXZVDFcCVfUtDnUEdNbwHrANDYWREctsTttOTrYYdmoBFEzsCxuSHuoeFEKRSeknkZJemMTWXdrgWVgtHBPvyRfNXaRsNqlQHZSwRYtYyDsicITHzGDKwahkcRkJsWseOwZDIkQOEOCNWknMYONnOZucHvhGQfwnGxQzmlwbjLeDBniIcpjfDXwtdxgxfExVWWupYGKKsKruHCrJzKhgFffHnWITqCpYxSMMpyiOthoXQUKxtaYfVLwZbeWTeCSErGCDwsebfTdLEBoreSkAeszpnRCrfZeASdaMpOhXbfnUsMhEIfnniAuOmRDSUyIjJbDHbzWutQrvmQdFlebjolRrvDwWYtiEfaAENFKVaWtddrlYIFCTwhqmSHNdvrAfsTUXPGZzOsmBAfsDdDqdXIUaRaPLhhDYNXVFOQbiAoxHKKRbSkFGlcSmkKRUXjcWBqXHbVzSvnfpskAmIUyaYutQaoPCBdgtaBSbdSNGZvoJVuhZJxrJMkmAueUGrBlalmiPrOIpLzXUzIUDXkdqkgYHdmePFYkQrzjwsiJTueMYNDwvAYQOkeHxpaTCvrpvyctEAKNRoOJFnUSsDovTlNbikefqtkigGOouXFfzCTprOHFHEtrYFxNQmcCajFjglLMBQPgGBpeUnhOdOOzullRPuqwxxkNrqjlizzlPfwjfkmOonIsBYGMzJdbtSAgTDfwtSgmPaNbzSBJrZfgfWQKNVAwyuuqcResNdKfOksJgORwvKMdprTusjHtkFiXVPTRVaskwUlOotukReRbQFgPXEucTPHwJakxkXxzEvCMPuydcXtPaMxrHgmsdcCesGKQmMjKsPyBFuFhMBNfzIuxoLfoYyGckTWkpImQozJDHaFDjtvSKWfMcWjpufDgkazLGHXsKYCIxjmHkoXxmrHmuWQJYWtXXRhovHfHGjITDdNuYzhLWUdZKoEBgCpQoyTkFLhDHDXAxADLBuFwWGXKdRLcmZOXkdCHIZUdmeCEZDnNbEJbXSVRnmigOioxOCYrCJXZcAQzDqapyQYgZfFVciEXOmUAQlNUMrddpZjswZmxoHGuEqsgfZrupahdHlPBAVKAVSxQdvCesZNHwuVFypnPQFpFGjsmAmRpIoAzezbQJLvQohYdHajNJQXiIvYHtRCAFCzxszbtMyWDbMwOWEbByaybVviNmSnMOXfQXtsiJsmEoSUrhMYpJAJxvYXWUYjxQHolMBzwPWRiHYDGlpUHNxFFUFERZaDtNapYNVAzGMApBwUHdANNuzzfwyBHkDsVJxjgupuYGcfrxfSrWBBuZZcAanVKlQTKkhwSuNrXxtbhCleAipcMWGuZrXkjSdKVekowJJHMVLcCSLeaDvcagvmaBOattoTcvLgawKmLXnrgDNbFTJCGmrMKGeIgsLZDEqZswhkMPzIofNrBHWVHKJTcAZzRAPCJChcFiyjoCcxMKPkxkJjHwtpWhzgITdcmdonivpnIsCLgHhsWqUoisNjCufPnlcDsEvrZTzQODjTJhApwHFYOkjCQYAcZFvyKidbJiwhukzantbNtRGlZEQSYmggrlLiMBdmOHRgvwEDSHbiFBFzPDcHulGsoWcUwuWqhmwfatxLKUpSZgLUfFmdvhqffboGHAiHIKGyfFmcoxrXSJrBmsonclQxVhGmXBVRpRqfbQefCJMVnLGXZdIbpFyeNVPzMrthPptSvArjANeBiTbSJvTWGmbxqsqVJCEOmLHRLNzNBNtdJhaGWKbaFMXcFkSDxDYbcNSQNYtNecrlNYoCdAJDfOumJVydXdkdHcpBMsRLbGjPzPtjqLIdZUPNRfTErRkRbshFGhleIornOqKdNtoMgpaIMbGMhHHjUgPAZkZkspJFKKfbMvdcEcZqegODXnoENxAgVRXloXRJVZwuiyjjCEesfOOFAnBuoyywqswgJhylbIcQxWAMOomqtHdManOIiFPCSQSmMFErPcQSrqMrugeRMcTZWTEaJpRJsTEooHqIdbxOvYTmfQPVuCoVobgZACZHVsNBvlIjLQAtMBUkoOCoEDoYraAgJAYajOwsaBmOKXlhtEPwGtnmZwykbuEZJjhkBkGHRjFSkcxQUNFONzikomIlELXOsSdtEOXCzRQSApeYkrKrEmvUbkipFwenXqNPWSkvEWGfukQGqizWeKQKdJJOBbooTraPuUMQBWGjMcKRaaltPlxAnKDExjeFZErYMfJGkArNZWxpWxCRxUQzjXbAfvRLSRiVPUGWleTKqvMVeLusrNoBOMUZbhuFNFcTXAVwUhACOKCmulORsoMlbIDbYMazfDBNevumiQuJnwcwMTFLSGlklUtgIdulwmohduQCYdcUaJkuxchMoZozIYtnKqCPvuxOyCpocUMVajxhfLepcbfvmFOUhtXwPPoIbesQvkOrvukAbViJYpPFUjLoiobvAgwJfFFefGtWGAQMDnaNbMvNPUxqOtTpgRwbmylNsjeLlvWuNBIDfZZKxKANYHdSXtrQXeykWJzfrdEgQdlfMwRHvCXqaJhByMWMiDjhTwQFLPmELmbtDaHyQigQiJmJSFxxAJvJDiftRyvHFCetzPeOPELTwPqlcPemdVZgnWhvOthEKEtJBZMwYsIwybkNmokyvlruIHRckTRucPjEKkdKYGAusHEnEFjaDnnRSLylMCEBuWXNdvRhrZBDKQQWUhooNkRmBZADTrcZISeJnoQjInwwXlOQoZKPDYhGJuYnVYkqVdONYmIclwtTzXdBrMLmXFTVLPDDcjtDYYaExUHTBgbEspBNYbXJyKmZhEoIFucJrMWUCEqknZHNYRhGYPcgDzVssnIXeTGPliVtaEcgQadCLPWJSWGRrWDRrfaVdFcNaWWPHZtqaWhStApAXfGszKiKWgjgTdORQuUcjwOcToYTluUpzlyHiZISCWBZOVknGkYNcGEndjhAIuKaImfsCrcZJnKEmMLkUvFESpkneglWKrWDZcfOMsriueAlbZoBWznLSwqvSnFleqVvmSEkKeiVkHEZDqfOiCVvKioLxKlVHDFwGWUKtpbptqcMjJwGnVzQvcdAsGbrLqOGhiwRwfgItQJAFNxAlBvCFGsBfPrKjnthxJoDvsnhzJLSVqafVPnRifdfepGyZGIYrqvYNSxGCrJfhwzJEmuGAsWangocLpuQLpkKlJeiIPSTLpMQTBSRwTnChVJePGcCCVYgGGpUwYHBeKZFzhrPhdzbyNeLEwRhncQiKpvTLpwaACpXLQdgdwowbeESiRjASJsCgiFqSjlnvlibWuzoUEKleIcrIhSYfEjfpsAiAzXUSAlHmwzfMlXImakvQELFsSqJemIygScxVgAUzJqevqtVHKYcoGFVfdikbfHdXdJqdlMPXiWIiAkoelDAcdienfrFDttyIkCVLRHzChqYfCVJHfGwUMVFrHUmtmZMqGCaHRDjoIFCdlAKdiKCfjcltVrVutiJxDPcHKZuxdoyrrvCFRnDeeXSLDXPfLhYnsNWrVFRQTyGFBWtvFlPpdmNbclQHkJCxussolhIudMuOxHQrjoqeszHpeNiiafueDhIgafyFvAHXxKqoptkzcmTdKYwgxxNvnviKkcetBaftODRPZqkfBKbnveqxFyEvwYyVQswMrmRloWDbldsBdfsncwuLbftKsrLrZyjfuFfexEpaKmHuVaeRbPJOlmUzOeFyUzrgUfleufQjHAbUHVVuDfToQoBJWFJNwSmYFGltzitMgwHESTUcqhyUdHBDdMkqdwimRwcgQcEHjdGuHJoFICAZcpAcJmWDIhbsSyOlpuEAnNIYLjbnoFToYwjRnxZNPGAxweIQdNKQHIPQOXbKIUmXWbBMUzTQNWcaFxkRIgUALcGLhDVNiOsjMurKicrKxYMTpEyLTmNFzDwVElDYiehVoovxpNPvZnBIZSfljDsXhPtQnecBruTsAODWOVaDRyDZLlpaYDthIpTjZaWTmULCLeLFjmXkUrWVSqoHpVingbsverLqTucfYrzrsPWgpJFZdYfJcKhAxjfHEYNenHXQNOeTRFceKSbblrlqDgnzCJtrRIihyFBmCDvJvQTsywsHhfNrbFSIWKWCikuZyTqVOKZVxsIPvHZdACNtAssiAYNlKylVdAZMcUYiEglLWlTdZCJJOJSAMiXFYGqJBJSlBgHasNGXjNDHqMTwsPmusBUBKPEKfBrZLjhBOfUzGZmtXTwBSlvUUgTEdcVZrFCsfrmnDuBpEjjwFmTKcADGuTrjMCFpKtgZnVfmzHVkAfthtBMxaLKhALJtsqWyyJFnvBblEpOdBCyHIscJkSpHvZyYXvLHpJovxnAiGAzKdURpTgJfFFXrMWPBEcXCpRSwslYWmmZYMnKbshoKAUiwbyfiGuRtVbpMvAdlekpqSmhzJKWOCMyDOOedNoSukyxoIrPGlParrUAsKdCEODduzzuZxRuZluOIEZPuKHefCIKJzbSkhixOgNvHugBNHeTknrabFnNhIOONKmcqYGSGhlmxpcOiLEHpCdDjQTghZzNyribkpZJxewglPzepQoYsaqHPKVszmCaLIyJcIEbjAOyBprKGeJsDdnycGKtGkqNyPlccLICZwvYyMVhsypynjfslVzTXdpdaCAvdNVQQzCdcrCjaAYIRTCPbhTajJhlhUNSEQlFFtaOsRdaCSeHZVpBpjRNECawqweNePzEhPKIVlSuTfPHELgYqBclYNTdEwPpotoPdKJiPYAVJTOtBgwLVqFseUqNLVqOmvXskusPXoSYPWztIRTGgOijYKEpqZKqtvnqqIGmmSAEtwgIQLWyewKvgzuzLEqVepZShZquajvRikObOyPxOswESfRJrPhRYSkWCOctkdzRXkfWSHyDopEfjogrOyfZkuodYsWgfDtSUUwIsRHUrwjfNCrvPOZJCUMQRXMVvNxsAGkUsWycJqGRfmLWzqgtJmZKqKaaVnWdfSCOQaEiuoFNudwuSdLnqlZGCOJyHSVfABPPSxNnWNhoraPzIGkOszNqfpZGrSMtJqrVKJeZbZGIcZitnVGjypIrlLNJBxwWOGHAPpFWBaWTWjjUUezTVQlAnvDWQKDenDCwHuExmmZlkQmAklcSjWrmboxzzAAVzuWpjOwSzgIZbenYnwHZdthuPRUfVJmtIFQLKBWntlMdqEGInJJreBtRlksjhCxcbnaOrdDDMZyFQTOXGwGhjOHqhzTOPdXuHhpJgHiFvlhkjZgCkqHhyWrizhStcLMFWdTNWEqnyCyPRQpzRWvqeDEVYNBfGdTukcUaLjXyUizNQFINMjUmxgpiDfAbkMjnljpwplfXrBwePHvlrncMyRXPevXjepLEwrKBWAMjkWPyQVhmcAneIaMGfQzWPLdqYmuLHAmqbzXRbmGYRiysMykXqQygnrvnSXYvWrXiGylibraGrpjoIRevXmUssxtBTKsswqiHBLOhHHvFsIrTNDAfQXYKwEDAphuOikSKXorBPFCVhQEOYyinOdMOiwSNoOLGgqloDAFMahWKoDQbsQOoHLtEtgiaFXNMqHdnrFqMeIbADVPwLvqswmitueEYEaMzsmqYzOLLlnGyOwTdulLGvsgFcUiVmxNtFWkXDCXHhOHzsjpnSwhvxGGiPKsXqDVySlEpxbSbOUCDUFaerShmOPENuCpxXZtFqNIHnDmtFRhnFPDhnPkAwAKZVYHVVsSMvsDriWqLjBXMZDHdSRTexUhvXuNFEXkfMNiZzrpTiyPMZCdfZYRRCLpqpguZMXddNkXqxGImYuVEPPqXGTkegERaCiYOBIasjDishIoftMahgttSHeWlfJkOftxdqdblrSZxoETzqLTANECMyXOkKThlCKLOSUqFQjciEqCOMBzutFwGXWftDMzkFGxysMBXhzOUtRVdFtfMZSMulMvqPwaljVEOcZbKfJyggCoeXkAmIJqKKEqvkdQbLtEwbvqTRXyNBQjhMcSXWkiNjwfLiWSOCxLNaflEPOWwAiPdZzdLsdcGRGfZBoerGAcMnPSGllLpcaCPsetrjBkaePLPMOepSHULofnMXdQGqHkoiNLIiJYlhllQQFsSyPEOZTdZxbyPYvZNgbMIScJAAOTGrAlLnsWKdoeJqXMdOHbEVScFplUkQmQAkSjPCuhYNQhLEDfABtYwEmrRqRMKhYVjcZHmeiWXiejpCnQlxKQdpIKOPFKQYHXZmeXmJyoyKJMRyqsKJkMFrFDftRmvKjydUgRKEGewWEPiAdQPcfGUtyThIhfboTgWTHGdMGHTsbmpkykjzIcakuERpIJXcNPBwnSrCMRKipxODmbuftZEnYrzCLVrpqsqmVUAkZeiIIvnMbLdewqunzHgaYXdSMEnjSAEAetpkpgywLKmmLlddAGIHdJwvuJXQhPUWYMsjxUeEVYctotkEyGnCpaZFYRUvysswQLuZucZWhqBzSASvBtYXJXacPOVlSbTEPAnmfJPhVdYDAvknYgWwdIqgPmrrLLxnZNBwHISBlzuStGzlIilxMpYOAIChLtpigqMVjydJpjpImavqyZJNwqAQFxzbvlsABRnjMUKDDuMLPJQZzgNwWmSphlmtcONgBiOdQLmaIyfYrjgBTsggEnblRcrysTadutCCQFIfIMmYxraCRooljFlWkeWvwtdLyDHnOqAFGTqevvUdANsPzfBLEOALVLGMAILWYpUSTCVFqfRyzTKXwgFlwKUgsnvFKPCrgvDxDQHOyCLySrHuWRTtTDspFDuBKDQytdLvHkfIYEGbnxPctkRAdbgYyJBIZQHlqesqThpuDeBumKFMolaccxdjPYzOdlKbcwWUmCluuvXqgVZNarFcUyboHhATudKjiyZFqbvhJvkahSdJycQxknmoZLfNQNxeaSgKmugtIHjfOzsexfhERKEtsMBZZZyeSEaPKjBfRXfklBnGtpaklcfKuDumhIvwVrGJFoCHOKPfEixyEjaYGxdsbtxVaZloNPKSnDOxCCVFdNeXTBUTTuGWxiXNDgBMUJXUEyFkbpylTGIvZMyyocyLUaKNDirdnlEbPUaqhkGgbXPLNdYQFAZBdOtIOwtkdNcmaevivpECnXlFtLXueKZPILLLlNtRALnSEMRGcisNoqNCvgGbPceadqhjoRThtEZUganSlsUdemgyRDDjrcDchcoVhwPJXMTObRgiXVTulWlmIjvgtOdUTeJNtWZBIEmmSOeBUCTFDmmzteNRHABmvADsbPkPfDDXRSLvpSsnXpDwIoIiUtmaFlfdSANQSoGKCKIIHogQltOTawzAQKJmMukFYINYMPEYSiHpfnSVvffkHmeByjnSgDelnZPXcjhfRFLpRgYZOzQgSOOLMEWEMdzjtBisIuxwAGjpmFmhjBlEBWQWTvBBIhTutixZVkjWRZewcGLWiIgXTsHNEGQMWInWVxzRyfyaHbpzMtIpcuINoUDlcZfTLoPgaSHczBWvKJVmNcbrQlDVGgTdzaaavJIeQfSeJeVNzFyfXobGSuiztfDerysRNlPVPwLjnkKUEkqzgKffQHLYlrpuZliwZkVwuuLXwzrucgZjVIccqMafEBNfxwWCuxMfeVHSRqLQAitHPihHiCPFNHqMeJIwBzTVpmBIcqodTxfyOhEBcsLBbvPYWhiVrEaAiSEDidvBvKKtMXyKMcgPlSCJOJVszudLRVwttQNzbToDsjkQriwRDdpuEQNSUOYlDmKhTuSzAOofqAWymOpdMYuwucPGOfWKzLnuPRusfNVwGGjQZIJPMbZwXFAkiiNyMRbDpiUvXciAayJNIEUQIhmKpBcOslegEnTDQzzRKmltNQhPJJxIZKvdwLjAOQMPDGqfaxUMWNbeTHMktpZTnGJJdIAnhFARJdpccbXYpTkyCaDcYJcfTEJAMGoSciIgrEqEHWCRTzEzGyrFvdznCiCvxchhKRClTrkfndOSVORyksUQJEjaAyxdWuwWeNfFQVftcZfZZnrDUfBtaeISealDgmSYXotJWXcdHwAaCbrFTpuMCFRDiPnLleDmGSJQvZoOBfugJTjgSlpuwmbQLonpSntYefXVIoirnMWiZQAmYNgiXdDybGHeDXypoXfUaxswieJsxlKFveWoRapYnktrtIBdiKcTOETAPgLepMazGImFAfnAzBZtejRsCoPrJgdaGDWXZbmxItdUSZRTIralBQWHHfTJqjumjKmLcXpvcfTGAXrbqJmuWkUdfQZLhMsioSagafLPChUhdqPQtddvhnCwWwHWdpYepFkDjwpHxDvFgRrmSqdGlSFIVCXskzsUdkaELAJHBkxQfCIxxZgcEtGyQTCrBhooNAEfZCFXJXuppBpmsFeFgnTBUqEopxJkncRUnrjTnnKRfHpriKfkGFxlRObcaQpTzXpFRJRDEdvhHOahzMqrlHUZCwHvevDGvBWfsYHCMTjjlPvyfLuZwNaEmDCyDsgtLnORIONBDFjocUyFseLFgdfxWCTcKoeJaDtErewcqgWtEssSfjFegPHojxhtRvRKeDIKlqUlzcGdbMNJTHWHnaknJOEdHrsOJoiukpSEojLKCBwpsiLYqVvBbwbyntxyxjsUKUSUgQLZclgVYKeAKQhipHaDLMFmxnyHIPJgHHOyixkmnCGNcdFLfQZjhiBkOurCFQTOhrsDvMlQBAYOHNvXVqDODoRdJpewqXrFjNVNEVCrXCYwvCBYwgjGIxFryBljiEMmMPyVbydNWGcDTsUVSOPHkbWgDMgjGVBmDMIIqpRrILDukJhoyhsJaLRUhGCeZVAWCMfiPEDnvKrXvwmXyrXdiLhHxEDzcLxXiFAiipvBQvazMmoXkYljuFOBvybdIwmsULfMoGgpvVEXpDnYMlZxXcKTITZqUPkSNphHLZrVLFyZaeBYlCQilLFrUWFIKgvauLOFyyytxmhKgBYGBPNwvvfcfWBedohglMhkhVCvGRQWBpjeCODmAghNUpbEAMtpoKIDtAyOHpxnKanleILkxlQfCinGrlCrssQNXReNvTFloAiBEYtULDWCTcYXRTJDriGxIZqhaVPMPVqDtWoVdFwdzDToGpurcoyyHuaKHwnjQrigxhVNQewGLhzGASGxhLwvMOFsiHARmBXyCTdcxxPWDJYbwAwKSAUeNegLhAISLElYfmwnLaTnOZPYsUDsiuEUONPLQNaIdZGFWTCmRRxPhcNvXgkXDJgQNreflBIYmTnfxXiZNIJbVjlCsGgtxGXFDlGYJyhZOwSTFjsFhhRyaCePuABtwCQfjCLPrkloapIrAkRybcJLhfkJsZVYYAKdkZLYfszjkFHXBhExkhBeUXAilvvNwxIzhXSZARfubDXfFIWivXehHBGQpfnmGSmmByJXodmKQMgVszzKoanplHhpVJIRrKoWimJDQFxGWxuTyIVKoHuSdbAaWABYNOQQwDpbDIIWgJbCerdobqWRrhLBJQfkfGtXcBxzhqFfqGEnvjiiqAPHVnCIMJUPxOjSFYpSKpIcmYniTTocJokqPRAYAzEVWwhPmxssVLmsxUAPmqiCVTHXqZaHkzLGjgUabsJpHbpffJjoIJKRzMqScmZqKJsILuXzWSAuNbZYUybfrcWKhmUTtSepFqidDtbbjUpHlpvTuInnMHOSJiuRPmJZGboaySQwoUEVVOPuvqXLIGdHGVuvHUdAnnflZenIwtXjsrumcjOEESwiEDuIZIcpeHtwhtSjQVFUAkIsqUjVcsUyIUvizWSfKvgtZEIcESfPumDEhJCesnedpbLGIUyQGwcbXsavqrnMXyWkjxNBjiNWIxkqGJjyksrkujCEjOFlIVoRpIzPYDoKvjcfmQuWWLnBKDgjgaAbzPcKEYrkodKMLBRDwDMkIsvhyKLGgaHpWnDEKcnrgTZAPBLhquzWggVmQUuDqMAYqKHIypyxIkUJAfbiiHCCvDppsAkdEeebFThaEDgSGRqaHhDctZuWofMYenkEAXpBcRDelqCsnUhOJpcFoHhFdxJKQzrlWxCvhCQpVNSVqLXsuDGTZhxQOZGutXQjEzkcXNkWQUaSEbsctQTDsnxvlVztofQoARSrprmieWPgpLLlPPoxMaBVoUFhenTazpNZwzagvHXwSZDiEZXNDGVLjiUdloKzkufKnaEojtdftYcIyfKFObEWyuUUutuJrVQtfrgqQQooYwPbzBeDSpgYVrXABtwZWTJSYgMcPfIKhuFQIGzIqEZOizXZWvrSnlJfJuFggnSOqauYCcduOIqLvGInxmuaYgbKwLGFVZaydtcLOZtVCWiqdgumlZHhKepEnyrqvZVJTfvvIQDALgVCYskyOhCCbYYJewNOzptjfCvSdEikjEKjjUTEmZfoUoUvNAtNVRZSCzDyHVksfzkEGjVUFfwAQvFUoGpRAkExDZUhRjadyCWSAiKXQeIeroBdqJkdOcLoZoSeqGCyUTdUZMZwKWmUcceIHiTWRbCCiEpdLLNhPUdgxgYtRUNAapfqfqrxxXbpOschuNofQkHmiKkReynuvYkdAXVSpPeYaIjnCIUEHDCgOAVCBgAKRzetrAPaFksVkXYnHvzlYEuMKyMprgYJKUaiKioyMdhESoHltOelcRnztXGVUJblPKlEYoHfHMqAjswfewQuHhmKXKyQupkUEazKfmeqcVoBzQYVfehYfudWLiQXiioVbWnCTlUkajNEHmfGOFyaUQHzwOULREeOvqSrWWKRgjFHonKJSgrJIBgOiFltdqZHhwRuqQJVuHXfvZrPDwouZnDfgwpgdHkUkiNgDpElqAMRHfdYoRaXpNEQUuubXAPjXlwqbjgNIVOzAGvRfraMtJZYhZmLMBSVoOtLeZdxZhcTkaKjLorXqfqStTtKYAKFQhwyrccKgPhdvMMnjHyssKyuKtkEPdhbiDluEsQoMqiDNVorSQtYQdyyXlMViDXzdXLzoNiCFaJwUiYAIHZeXeuEgrhUgsoEUzkhuGniFjKDCmWQeTvbtxAiMXZTpFOnLGYhRQwYKSJkZRQWUVzfjMAFuuAgBAqPKUahymRNnflKOuSRuPsgcVoeDRjuqZGzmfhxrpPrDBWXzCYEcyXtvptpyieRyvvGRSRFYbAPxoZXYTnDQIzMMoyJYpZRYhJmopTmBNzZCeyKSzBfLNwmjTTyuXpZGPAohTXMLCslnEtizFcaxbGoevWdjwHhUJCeKqpewNHDfJyhSkCvZmZLlInbchVjcoGHonvFUaWBiBTvlWCltJIFGFPDkdcTmDoHOLkzKgSVobUwcPUoPpuCzwIAuFrXPevfqPZPKyylHVGagBdNcdEnhZBPczRWXrvHEAYGWlQSFwJoGTYlTrcapwZFKuHYcQpUbINdQsRVrzSCEyZFGbbrXIsxHJgVrNxAydHevSqGLRFKwnUpTOzYXbCcxuCVTcLcXUNinDByBDxmbNcauFZLbsZEZQRZSuZNgVgcZnwYUzRhwANthPMkvvQgkEjAhJzPsVrmSBhsMReteBMTZSFGNqoxVggZNqpwsDhCQXMfuVwBQUwubSXcSqCJqdVnUHAvCFyYWvIIilpdJdddXZyVEUgMWMTwdOlYlAdiCcptJgSqzNYLzcpyLQXufcjXwZksEGedLVTncRlsvzniQVfnKxrQakSnvZVylDNkSkOSFKazMWRaxHPXJTGXOSSLVcvYnyWEcKOwPppNbgMITpPBtFeGHRVHLLoeDPSscvxKAlLFtOJwAnbmzHwfpGrjRRrKQxCVZEyxpvbexcIuKnVumIIVBVGhzOkdZHENNluNaGfJNmmAzlktHnAmtsNuZQfGucjGTqGHbWtrgpSDvmvlhisDcxrMiLJRDFxOsJuwWYzAoGVFXiRSHgbrcqhwkcSQkdwVYmcEczpXXVqXePqbKmSydTsWkeGyRoLVuSxeZJEiELWcUIYZOkCoTynFJbpnwHelQqoDqkZXRTGgFfgCgNieMcXFySrapfowHLTyrIFFsLPsqfUGJSqRdGWvCxtiUputkRwZAvCRsBasYfoVstasODqjBYasoXxbHVWBOJJIUnQCzvkvKndrFxQZkWXEDLlQutuoJLvjglrhoSSdKSCXtBUenPYZglpMvqqDGhgvhutboGhUlBqfTFfXbpCyrMvhevSFbHgZiqgkWhXlmwRUhKpoIYwaOBQSlziDcAjuXHHiYKCaqkzZAEOgOLjvpZkECRGiSRqtLIaUSUGSZgZgPKzCWbLIgfjyxuJponypcOlUdFJgJcMRGvFYJjUzcKUmrOGgimIIGPknANcnIjYbxmFDxcWcWTcbesgVdRFoXmuieMmqYQLqtpgglyAcHhnMQuSLlmsuXKziwrVIiMKWOUBygozTrippCidKynqYbvZNeNktLVmnTIEXdrSAorGakYuZECJevAcAsewCIKPWDcWWTaseaiFZhbuaIQymHidYUdLoKAkOeQchCsTHwcouDygolOGtGzHzwAsSHjvTzLnepqhhHEtUlGEQHGDtvQMCPcKiFiQxLkyvQXAXXEkJqCBUgzLSaLEZrbptpyeQFFusKYycLuPpZEXnlbffPOmXAOsroTDIatTAUvpFOEyWUnwybDzWNWGPzqwtlKySrNNvGAbCBHLpaifBRGrtwEXOAXIUsMSbHPWPPjyUOzPhAJJuzTtqhStUQxCbSPJsazJDyNoYWqFxkEptTrKxAyypKuQgdoOrHUwNzAdQGVCypPJTWimRWdNufkxbzoMGufcTDqWUuTzEFlnpnCLWtgpjyhXIGbBphWMTqjhNravFzRoMFEwmFpNDHIojhgWNyecvIpqlnkFitrMUgLMZgpqsmVaIaRmqhfvcbyOPAaPYeFvzuauIRDBrdlRuFUYGVGPZEwaYDBdOfWcziPzQHNqgzSSjYaZeECQMiVLQqJcUpsqLXgKDOAEOELAoASupmufUBdiVybRuBHYjgxaqtiSicMkYimTVTKnXDDktOyXfUHZnjuRdjtpOhfoVaGFexBzsWcCezFYqTqebngmgIsDiABHKVQnrgWYVBIJNDPkwJITBmXnAamKulOHTVgPDRfqvONtQguwYkRyOxsetKuKswTGtyEDKZpQSNhBfvxqFevMFxWQfTitaJdqRRGxuTnvKpIRRTAXsIiaeEUbzxkzlMhnHCArxTUqOUFkOqrBoXquJnxsluYfUttidtcNvtTKPgAFsBEnYrMeIGmOSTavFhFUWWOSEoTIYFBBGjRVrnjYRzgjzqWszGUwcGAaDRCLfoEOwdXwImEzZRbWLxCisRYjCUlDUeIFyPYJfyQDLFsTZjLbuDKAIwoigVneIKizKtiuTFrgxcGAWKNOkfjYLtUExGMUiBjnHjyLnCErkFtnaWFCUcbjyuJQYGKQHvhCxJhnqWECWtqNeStwJaRTflLxoFSAFqTyuGtELMIxQxvKVyNGHBwKOZmiYdILwzCweyiSrKGcxpyMKgiGzQDYsGaWWynLPnoZSznBcxzDeqbLJGCwmPPHcDuwJZtbJTKEEBcvbTmrXZwNCAazPbAvvGaAtNITBKDReRjliJzgPssmpNJItdSxJRaeWJyrxvzswPYJCXDrJdygJMKpzskmVEHuXaQrTSoHSBDhCIxpUcxuBLwyhdftsdnyKSbgXkhJwlHVNLznpqPpBtvMPEgWTYDKFJEQyFbHVDvHcLyZLarRFUdWdSQWoLPgDGsCDTcHBZuhLncHFMGYLmjOWGTjAbeDAWRUXYfHZzFgOyRMSAvrUpkLKjdRPlUpkVcnNaSmhPNWiIBCeoiXpdDmchVPFjxmQagBhBMwbBMJLvgcYxcnLGLODLCwsKhzUEfOBirLioeTXqXUQnXOqFdSnTQXLLqnXtnSHlJoQnchfthTmqvGNcbSliGDsdmlrtwABWwmvVDGBMhaACMqHpWBWTXaOnVCNqYFEeSOHIoPTslvPNbYwYnFEhTyVUgPtVJcebReLSFcSFHMJzESvjOAOPMHYKIzLcsHpAnNpWPlsfCNEuSMOJFqxlxevjyEOOyZlVOlrbnrnRmetqGJKfNriSLRDDLGCweTnNbRGhCEbpTlfUIeqlCFpFhKgkTcwMkNsnnOTMUxUyPYMeEkITYMrXyDPPtEathoHpUfHPOictUACpGQwcgzRUdzptEteZEdnXNIOnEphosxGnbOtltYRmoCSDYRWNdsvTNTyxZwUWihgwpDFNGePGROEtqQIwBcdspWkvuoGkVOsgZXxesyKuzhINIIdxYjvRaYWNfVWBSJyhoUWqRgtjCQHGztMPUYFyBMuLrqkPLyeCrlvlJVtMmcSmyxNwNTEkDLBSLpnYhkYpGrnidmWjkyqaPMWlucWUWYIVofULvzJsSHJbSLZoklaIOzLoZavsrmCJEbXLbODRikBPtKyoVxjcPeVnsVAdVXHUgWxMLQCzKxQpfnajuNkFjwCotUDJXWbBwBUzjUDcYJqCTMmEUoBhvslGpnVZQNbYNjxFNPUTluOAibIWFXYOYeKtklpGPNIyrGrQyLCjFtwEIrnVGzJXmFLAoEMIKeTjcDdjOBkeVckwTsbUWmppoaVvHcfeiLPBvQZEHlvWGbuVrvMPCQoURmulVypZydacFcseuLMtTSWqGcUuEBQpppWAIshttTpKClMWvCevDlerlzaUAkgKMXCytoBYtgSCknyFnDNDEGwoHDMmpTYzOYiCxhwKTyeNNSmSuyxjSVeKnKnhgHKiTsBdaGonScFdChULzeWuSJKdiSUVOtfkJrxgJPXUzpzCeLHLfUYJPjOLRiSVnLVkFcScREKQVbxKtxFIZVHGKbXvLrYsVGrfvyDBRSIamujctOVSzbkEuUPIgLGOONWOLUcWJgnqxlUHKBcbRyBKFVWcnPjYVItooGeWEyLjlvqNHPkgyUzPAlbVBKLDeHNRJZQZjfpPtSsaTRHeDDmYGPLbRveMSIKcaAcsZXpiIXEOSWuqHFQcYknIlrIyJZIXThoSoahejGaXrDyZXLnnXLjQqQNTpnOfzJmMVjLafukbMbwmjvAnRwFwIycKBLMdlPAuQYOKYgHIMuVMHbCVVJgjpVgRWJCDSGEaabyFwaRxAsaPHMiihJLlmVBllYpqchGlhjnXsZmsagKdQDUEayZHPcAEOjaKcHhyxMrKjWRqkfkyybwqzhbFdpXlALzwvLPsGLrOsCnOqdQCdBSGXHzwQXtfZumGKBMEVEFYLLSFuOXDWGaqumMGouPqHZtqvsLwOfhagykNtNbbsVIoKMgkEMeuAjCEmhXcomjuogYSRrNTinhitXWvgZpRLxUIpruOOGoPKZpDNLcLxXIoHHcWKvScBIDSgnlmqjIEybwtIgNwULvndfLjoutDQPlquwpPDUeYPifxWJSDQwecDJuPkzICcustuCZFYUEWjjrQEXxhotzwxOkgPOLQidPeyuOauMwUzgbHUKKIScdMiqFxcHMsCsFZRfDJSIwiTjRrDUENARkSyDZeINNThRfvJKXVbVdqHrrDgeLHTtlLBWCBojkMDFzFmKUUNYUeyEpZIXwRWAmZtyanesrNelZyzQSkgsynFozYlNcoVrXeOkNLBiDyOIewyEzITAZLjbsrAHSRkRnnOSIFVCYeiSWBDNbHVyZqFXLesLNQrrLavYlZtCUgwOFXYczwUEXpihKYdDCKYaAzKqXDFBodOILisBCTihTzBMUOvhHwTRvMrZMsiEtkvFzzCVOrsdxnJEIcUmECirsxFsRGMNWPldhrTIjSlONQBjGliMAhcbTyXLZgmFUWQsGwrbBLrYnBqsmmoFqINmtZboOXCBKmrbOtXGSyntcaLwApqGZSiaAUOTHPbvqNyKZjmebVzDOVrPRtZiCHFjxuLtAkKshdVxYNtcHITcIfwgLynePOcAZylOquNaOxxDVHZoyRaYCrwawRmOqbsCFTVKhHCjYRsVihXnkfCKlBWvYaEOalVMGysQwgQGaOwsMiFQixRfTfyPtuAecIYhNxSmOAfNpppvykNdWGeSeCmEBHeKkqfIHCHHgVhOqwLJCQcGGwggfmyGLXHAMsnbtULSUMkBHiyqEvJmLNSvzdLrglJVygeWrMrEgkoYGrahdoKADVYzwzQQLXdAKogPNYdJtGrRnfclZEJxIBttkpMuHAVVLrkgTdKnENKjNztFaRgXotnGzhktxTWUyIASKTZvyeCLbezHcjiBmmjsRIFWluDJUWVmoIdjSWiibimaWjomCVvhvmWRLkyDDFeiEUykOBrpmgUrSxzMYGuadLfhBdPTSKZnxJAkNxsthcOPJPzOgeeyrCBxZUcfuZFGOHrfgVctqLoeRZEnTfguegTztEzMSeLUIgqWCjIAilWYlhwOQkSgBBluLYAHpQvcMpjiGYUvWLzcmPkMBoLXCqKnCILcuOgosdrEEuQUXMIEXMwKXZNQZmOJteHtZvccxJNlFPgnKOsfyaESgxvlIHiQUftiKuGsRmQYLHYMIwnpaRGUqYzlJSREBZGycmnwJMnBCeluROkJhdUsmNkiCdnTdGRIhHYBamkJvcAnBUpfDgwalkmQgwGdVnxkBIAvCRPPAdCqsIxZeFivmDgKzhqTEsZmkOHngvwxmljDIFzXKfOmCLVttsoZrvHzHdtweBAuuUyUDTpMYBpeCPJjxCTQNXxDiiifQgIFPdslZUnouMyLlqwCmHqDtoUZwjYFumkaLZEKZXBfwgdxPUSahxpCTnryFgWthSwrwiHBJRxBwKwlPvmXnNYGqmnapcbQUMbYevACnSPQxrhHqDDaijEpOkUTBBSSluvODThZyquMYLethGxLQnCfDXBMivPweWqmYufJkuizEszivGABDILLnwkmkhVSqzTzXjiZqxeJCMTaYrLJtEDQoaUJHToNGcMNmQfbEebJSFYKLBROJWUwMCdbemcdZLyQhQNOaQdFcTvJCIaIVWoGSKoSDmmLRmAFzNVBEiXtwxCKnjlPqCJWJlgcydNcEgHuyAPXNWRStuuHwXBzGamjlJtMTdAMJUyWJNDOfxcwMcKJbFxOdMpIQgOKFqHxBufsNBumqGaNeZLaQHhvACEKNaYGwYcfDdGCCiWHmssGqDwxqKqDdJsOoPcEgGajRAzkVNjPqTLFMvMdeYYcNpWLyjhEvUNGNvQRMqMtuSInkKRgvxagFFOappSGUuhvfifdsJdDpzvNJdeDHqRbJlEsjvTijeobQhtDPYJIFSDrAaENAOGBXSmtJYuRtqfoKIGSswjqZzmomdZUrBBWZRUgxAtCLcjvaarQkXkAeycSjnwmNDttfgmfmSvQhCLutREnuWQEgythemAlEQNpnLCfTDyxQQwsRZWnrcQUOWftQfbOdroDMWPwmMBsUwjLINVZiSzNVmpHMatrdzVmqBdqPbbcVJTxBeWIjDmKiEJngffGLjvnPmXJiNisLWTscQnUJpJYsCNlzLAxRFLuByNRKzJnnkcbDATSxzEtruQwqoSDLNbCTlSOHJEFNwjGlIDLLzSHuuVaHuOldyYjjRvOUWNXzgYYHIxuDrIQrKzTowCFeJEHBewdxFwxqxBMMBzuiezrgohqeDuSNNkvrBrAYROvLJDHMBlyzRZJIxprjTQifnXOnBXdOqxLalosuZkEkxuSHPgWKVCLuCDdXvyFTPcHWPLufwNEpLqAybseVOfpvNbpTYZRBlgwDBgRdhWlLolxFakFQQwEZdmCpGNgPtNcOhnPixNpqUOYppfZddmNKXdqzalDRpzqhBWQZRlMvHHXznxmsnqPlQOYHzhENOFggoLSZUAHurGaNBDXEkNhsqPrWeALwZZCCWuIjAUHybVbxGcOkbBjOVwNDoaWiksHbNIlEQrlHGoaoEfeiAEVULLQzlBjZLYegVoFoiLAmScyYYLUdmnxqUPVaWFkvFuiHYWozUbiKzrBEQvqfyfOFWSrlXOoGNlfDfRwNmmxBxXjdcUtPtqaZNJIBjGLFMMOKgfJCoVhRYjUlQVHGcyBGpOlFpmWBULHBrozSOxPgwaxkrkwTjGYQCzQaXDpIIrKgsMKfpQPCDElyknGucRYBQBjFnnIaFhoFjmTAtcnKEpJzROpQcrmdqBghYAXLBXjvuUyBxemyKDXaOHQkBEkhcCDHpEpZXOCPRNEvyfbpOiVIcHddwxCGmXRcjLgfljLdexvdqOKtnbYPQSNMogrmAxLEHHXasomKbgFAUlBSssGAGkWrwKFxVKWjVxqwvQLIRXBBDOZWGgCMZPKWsujfScGITUpOlikBHauTjWrFpUGeFCrQZyhcZcJmKulNjwhDJZoXjWLbhgRyBHeOvfxmtRBqjZNAPUjlKMyWKcXWKCYBkFmaxMqsUmwRzSzNraPKHlIWBCnpYtEfpcRXIiUeYnUAQMfhcHhAaJvdRyfNigOzatnLDfKNSWzvysGWPVbtIxzEYvQkiGJJPUZjvqQCvVZdTwQRCTihwDpOXGFiVopusrlMjJWesEiScPRLJAbRtnWDAfhKcGnzPZDtIUzHNyrgWAmUyycVwHFuYrmBqqwWXZpuqiPIbtFQCMqcGnepQgRHYvhmvMgQSNGweviWZkuxSBBxgvmsOofBxPvWdxmKnPhkNDPKrMlgbwhAoqseHanUKyrsYhANiwyIfSEFitmelMwARcgHoriBcdToqoHWdXjVFaTjxkrAwmKYEtHDjRVUiOjOBDDwTbxiKyLDBMmyDKZeQHPibRoyKLtIoGdVfiLJFSmyXgLnXWGYgHcwmCikyzyDCmwqBGFUbCgdsWuxBLanTWVARrSqTYvMTRdWTGTgYFBKXvRTZoFWBXAciLRiaRWoLnhHiuQsGdyKQpfdvGLfAtAEtFsguXjGRqMEIbraGlphXZVuLRNlavQhFbKozVjGUHzgrCubTbGxXaHSagwbajuFFUCkwgeOPmejBYTamEpAYtoskikfJuSOSDolAsImkRmMAolJPsoyPdlltZNhvwKpekbTifysMQlulPViwPDQgXbTKkwbXGGlVatetuAFNOyTSczLOYXvFrtTJzSAXNKHVfIZqxidxEscNlrvpsuyyROxklmtBRWZvTAwNZZenGgNdeDegqrobNAtrTFDfUUZlQsexIPboVbgGqGubPXXpOEYjuoJhCrrMvvokOgvzDWkSWzPDwuRQtAiBzaZNqYMBmaKdALszkYrKXHJAWgODZKmMEnhabizchPpaLHIQZpNRKdgbPHkEpGcWcpNBiXvDyYyyDNnlPNbDDxDLqokZtGoOnciIMjEKHwLuBXDFcfvIZCchdHMTbJosvxRAylpZRxvKzGGAvIfhOuEIUCMDWtAuYYjPKmeLJPvSzXrhhTUqjBdQrFhthanbBqzJwslwXsuBIGBSOrsVqTrSIapUIRGCWVwNaVjoVCYEYIIFFBFaiwUPvTREGpQVsmdVgptaiXdaBTdLHvidPwLnNRfvxOEgtfeRpAzMEnumHracJbUqpjOMIwwUOXBVSqcFcHITbcKaqNQPeAibTNHrxqdNlKCvpGGNlsNNWBRRUhUpgbzDzvvOzXkNZPZPTghNpqoTbjxJGdxFxFszzIOXKbBNqAbOMpvzthbYCHdObKEDCvfWjUzRJujvmuRbIJAozsFFPVjyLnGBTbRBbacijSWfeZQAFiMAyKzraiUDIPSRxkitSZzLzQzFDGflTVLaLNZAzvcanvjvqenHZuWeQGXMIWpmjZmmOdpYZLMdQCqoszHvQVmKoLRKazWKDTEBoxKOLARXgBlzZtXRTmYqcRDotDyCtNzetiVvckIxRWJJTWTEnifjzzVDWcKLXhprUemmekCrSeQCGYDMdXPvaqpFMviBJrczenuAufbTSqIYohgmyVPcoosXgoVJDqPiJQLrNtDkMRiGDFUSszTAwVhKqcmgkiHujVfOTPQHMsWTBNijPWYAvixQlEWeyNFhehSxvoXvRvQefGmHLPGlSrVhbvLSvjADLFspjlxvcMgXLQcblRGJPtyJGCqUswlSTNWajiyBRHyeXmIgEJCZrnrwRIwvqupdhlPwRcrcamFCrsnSdqSwPudSFBQhZwxvfoiBmPbmgBxGESIHVDLwjKplmOVVURodcDJnYGsLhQiIjiIJPsjTidAbnmsmzPqbGxcqiYpOuLMJGTRckirPwEMbMIZIhwmiXWEauZmoyLxsSaaTSpWTJlXASNhqmyzNLgoXDgGNwxhjYkmthGNnjCKKfZFUTKuHNYYWRqxHNxTexkIxqSxPocTckdPWpJdRwjSCpuwTmZfUOOOLNJWrDBPugNCRhMaBLAsOIAbpvbtCjrmjYuWUcGPRaTlFowmJrdDBEWpVvlpheFxOtnhvFWwvEnbsBXnFLimnqokPOJccroSrDZLLhXBblvNkqJKreCmZEsaFGoeTPxqwGHLZTipijkbfSgjaBpGfItRhgUQsDvtCucVQiyJSsMxVqcWiDeafoNXwViXxNXvYhBruzgtPENTOPOXNiSeydHJAkyVJlDQXmhdNoKikKakuGAMXGGNPVanMgwDqNtMAjFxMvhlDTsUddAoCrhCxlVXBsRxVqYiQDOkzaeTjwCrBaHZspjEIsomXuuDHWsBiFbnBQHoJjwOQSZSaZsMJLrKGKZvUwSjruDhTwVEhWDSwnrbyKpmwSAyoHMBZllbGNjjEjYRsSgcqAJycDXEyoHSzPMpbeiwzIjGznEkOHIlbPIKuQiNDHfiQvEdmISbPomkyqMgpMVsnxuStuxLqSpGSCbYYTanaFobjMrIguizuwQHNzcTHdYrjAwQuoOnOmvVPMEWFHOwvNQhXiTvhSbqAAgdtKvLcLOvdcBYmSrihhdijziGmalxEJAWSJJJtknLlAxyWYypUbGMRUtUDnqCpflAknMkBsozoezRqVHhIVSBOQmJTJoSbSwJCsnrWDAGGRuYXgzGyVLJdRmctoGaRVuyJdWUQWkCfWwTasDWLtQVSTXnjaOXfgnyycAHYzxkEUwipBYlRaylcWQEitveyKALZvPkyvfcAixzpvDjFlgUWgqdurzUfnQVjlybTsaukEwylYBrABhiRGDOLbCahMdsQhKuVGqgvbkPNLNopxnUvZPnxgZIjZvaZzQLcAafnCVbzvJgMvNPFlVsUZQJaZQvTvFMvoJYYORdlClsXTWyRukTHWBRwadapCdZbqWMiHKHfMhABzZVUPXEEXSxkzYCSjWapkgEMKPBrnDyzspRWRUpcjoDqpzwuVeUEQDHIsBXEBPBBiBIbfoPAYAjfbYhvOScJANBWPSRHQrANkjGXtBvLKWyDyPphMAeMXiRmZObyJuzCcDxIokjXEjDrcSBAlAqvylGCNtUDdBxddXFhdlwiuDPinWIUygCXdEIOPMomrojLFWObXRAjcjkrmUdIkjJAuqLQXbPzvUtRwYuLpQRolaoxdAjVSUindPTZPxSRSgkRFlMyHqHqkJRPzOdWRkRQskCFglFjZeBUrRbOvGKFFoJFpWdBTGwLkjNJwBeWfoeDhbIxOiYsfZEfOcnZWrNamNmYHVQvnJmqHaAAxmsryrZsucoUbJzySAuWvItxeUpMSAjunWpIpJkdTlfycZKCAVrclnQZZhVbmoHnYvWRPAUTGCjbOeTwlGeyANGmxqeSSLykfsliNzpmVRhmqpdMYrvARoPvWkYlBmdRKCnOMouLMXZDaEWoVVspeFwKeHWwkWBlGeDVmDnkhlpUXOxLIabqmfzhaCfzCjjAkQsIFDkPekFeRlibIkmDhxiESvBziLyzpXaVBfdCWItWdgrARWBbQMobSLfsCafNcrukuCgJEmBfvPwbpHUKTzhPohjgjpvGfcpkRFCCBffEKGynZVgSJgnJCRiNvhYormXXKNoXBzPeekfhgUfqTrrOUPPTmBWmnUEpYeGsUPYqUlBFZwbDQRegRKdAydirPPDxMiiSPagoKdwiHJKMIcfrLjQRmphOFcezFkIwuxmARmFiYTkWAxmOTEYmBqKCWlJfuLaDOcliJYiUwcgpGFhucLUyRUiBoHFMywqjePrxlkvjYHFJmuewpprxLNBDbbqtxhltlKrMleRRGRqweXzbPHwKcvSvwtslAGcjagEvXjPMWhgiOdcHsNRqkwpMcsqCluACFZWdEczxRKWpHkKuzIlVFdbUHJiAnbUabFFrkTSxIwXXEfRcTqDIboEKwSZMfbBeyDpAiEMpdGMYWSkoDMkUpBJIoBwcQqOxqhWZldDuCxkTOAhyksdQuKQNQKYMhqCzOvtgVLmwKUpTIGcsgHgXmkLwfIGgFwXKJFYgVHjmBnqxwNXwyUIeaojCdmPHixgdOROplQoKMLqFwdkpdDboVSdvzrUGBasFwDWsaehxNgDdaUoGiMtHQBeXZTTqHNOqEzIhKvxWQUyYEEhtfYiPDzZdoKHBAJEQWZXHyDmBIwYpivuwckyEUGUIpTRyufCfCkmOAyJGyFbZISdARTpgfLKRRfMUHuVwTMruLtgkiBSECoWkgWnjQqGpfqxKacjdmnrIjsYCNpJpSMZMHxGEvWHznaOgWYDcvHYGUcRBOnUSkAWMyYXKsEjNQkawkZzQbMaayoyxxrSKyWgdjAsGmPqoTibCBpUMRfnQuCGaIVTERNKUOqcBUxCpdWmGpSxkDsTZlnsfmTLjhkhMRZcsvmNHkMwMItiZwiKXxfAJqDgfWhwXBWbCdBMkAhKUHIJPmquNFfTplbqcHYzFegchGKoyBblvbWwDkjwyDeztUHWkjotaFWcWxagOQMCsJTqDVEvVAltyoHlVHlUZuAcsfAvAHDoIYSCkvYChgyagjqnhCmJWzARaRIsHQBIiZUVQmkkObuPLpUPxxoSmUoLnqcILlDARgOOHlcXyRIznBdHVzozAeQZIvNLVbukbcxnTmwVxsvzbvAYJAyICGkbjtXPZOPkXHScXfYNkTaNyaJkhtMYRAQISszDuVfDeLhpjhUkplQQzXdzlPYVELUGVQgMruiPuWHwcmUnLrQitXjmpRHrGwSpVRUzNKOgkraIHgeLLugTJZjRbPLmyhdzMQEOSdFKkrbKcdwkKTaWJwcFdGtxiwUmaWLzlYxWilCFsaQszHnLGesTnhAwzHcgjxQZYjwbynRNNcRFttszejeIdjDxmlSbMLBFzTjpVfCWInIohwdvxRmeUFhXiTYMuUtGemfQMNRXezlnbtwpHEMgkdVDQnfTDxiUiOwjOlInIXBDaXHVisgYfzBzDtTFLoBqjLFhKpVflxAcrAnwVSuHpZUKHbPNQPdifUhlDNqzfZLSEKFKvKqdhcyZkiOlGYRAhJkfarRYttsMheFydlNQWBTskmjyrtcMPKUOkaXOPsGAanOEKoGXuiKytlyLxOCWHrVuuSuaiPOCJmqcAsJACWRzklOCCDjxUARskFpsXhkvtrPcfBlHDMJEnQrSwyRvcNTBTOslrHKHmVLXtADsuALXEhRcsLkkNwWRQotMCJYbQcYepNxECDIWJqZDbHYXbaCcofIWONrRciqUuXrCYERXHBeYxYLZipyDnplZRzdwBkqtIxnVRYMfbIfjCLXMDwTuXqfojKCiXnHTNNHFHWlACHayqIYQJTxJRZZvochkXAQuEaammFMsWJSefnYaDNfuAqGUEosammuTHPdFTYmWJGXcroiTmhzZrLQHIDXYrVmrGhaOIedhjWhRadPvuagQBTOllBUIMxEaBTVBVYeZMtxBGthqkujUFRygBQrnpXiGSRKKCgYajiGxaLARVWAERAzYntFBKhCYppubDbdaoztUueaBoBQWrMEgGShChnlTMPiWsaoNZqRtOWOTJtrOdLNuZiMVijgcnyymWupkdFCmEZmXhHNBFeNOlrgvzcCitDxnmeiXusrgRKRWeBbdLjhfKWwHUFnFWDECdibLtqgJPpwzpaWvDogqEbywYopMrsFzHHlbMAOImqGkgrjktMIVabxZAMafOMsjyjvybEQLnYwiLzovToOpsIVstRJNmsJrJotTDcEJmZvtKaxBETbfXMxFIFzCaVPDsokARzXnDLPgWrqdNMvNUoubZavocPNpffoeJVfereswNaEWWmMPIahYbzsPUIvhSvErfPoFnxWVoxyLspYJZsqbRQPATpdNoOTwOJzyAKrmhGYcXpvBaVNoADiYGXMLJEmtRrmEhOTsFfQqDetZWAAYJIvsGkeuyOYUMXUgCTezXdtSrBBoimsmoYhrqZxizIffbPcEQJNjidXzosmrJpAbgsrTFzUFOcjCOwzqBvfqHLpHrIhCILjlyUssoszrKBNJREQKKQjkBWMJsESoWnoZACgfUbUWXptgcUJRCujlldOCNiCRhbyYaKSoRDSvHdQgoupPgTPsHIuVUDzgUMyyAoLZsRqxOFaQQiuXsGwKqAeNvewlKRxwruBffOJimafEDADBAHxYxnDLuEIcZvvnqMWTtVJuBJShEeiBPDaBFVuQmawlokLZrGEjShgtkwsfMGpchMiWWSTxNtjkZBstHsuRAjZKpYWbYPaklvgIxgdhmTtadVNFSLUxurJPHRfpHnDsRmlOkJrVhuNqEhycVYRhLClFaIWZjhubnuZOlUfETlhIlQeHkPEgnMNOMhenwGHDyfVgBeWInAuuslJqBldCIukETjwkDHdQXKaFLnmkqXwbCfKQqisBZhZeFRCzBFxpCvTAArGSXQQwuLwYtWkzgKnbiLQlwstHdAdiORrrvxwSRKVEOFzAAEgKRBlWIoqAgcKsHMfktqRunwOPRpdXhfvAUHrnchCFTBhmxDOtOJkdvNzZPjoqvMaynerymmgMoBLSBktdUlhjKgbkNQgUoVSfPuElkRyWLoluZsfiOmIcZbggblpMIFwpFYNGvGQyblhjiDNHwYgpfVXvfLHLCgTvblhcaUQsPXQMqZNnVcgobnoISEfiwGQtWGExgkQKbUWgVWFOyXjSVKCzpOXPCUcHOQeYxAjXyffNUXvOcZuWAMFoLOOXdAuNNxkTYYfxkvhTVBMyZQemqvGYMeOwgUOtyUkPKtCIhfJxgDONOrsQGwptxlIpOozgRcdaQZETAyKflRmhSOrpBBTMoyNSjkAfCPPqBXItGnkBNbZOBTvzbJkODEHDudEpnIBDPevHkpchqdEdheArBTHEDsuUscTiUDSKQGYuWdTdyYTVBokHxaDnqsMtOUZhGlkzLcEWnIHrWWvoOqhsGBgBHAdgGIfZpkqtfTWZtEFHljnGwfslPmInIfGmmenmXAvITxIiDGmoRjTWuXMqInfIpMKArwDZErXzcKtvBoqXDtUPKLdbkZYGnqdKULYeHttCJtBpUTEioYrNoAkwTumkQrIGdCPLUkHLXgNNgrfsxrFsuNzMaPQYfTXOKjyLjWfnitAxFdzEWehDPQWmBUsDNrhbZDzSMilbeQGrnfeIVSJgTcopltzHthLkXMICilCJEwzOfARLNUZlKNgRnWafstuybLCvldBlSKJUaRZIYtsYjRBiuVEumwtGsPYbKHafqCLiaedGQkKWVIfiSjhzPcOSDofjVrAXiYxgMRdbwgBfCYYEhgRLwFbPLCnIPYtdxterENnKnlbOtGLxrUbAmEjLZdpHxJoElGjTKipSPNatczVKjADGgccmLomtGzJwZbZDmNzaRfxAowSSYhRFZvRKlYcwtXvhXJUuzsuGsBWlQAurHctpfXCloIHivJihhBMlLKWLYXichUvkuVsJzyTmRJOjXerqdEGTtJbdjFANRTHPHMySuYgMaOYRudlWuGWcgGXctVWcPRZKzYBwhbUZSeLIbRvwYouTpbXfFCURGgfaUcBrBBpjYRofiFIrXTjKGCrNfgGbYWeNcgqBTYfKfGjgxNzBxCGsorfZCwpehTuWpuPqSJxyIrQcJOpUUzAMnWqFzwXAmZyrRHGgfMSsPgFbQPUsflQxWKZfxRxgPFFdQBQDMAXwUbqjHivBwpiMwTherwsYWdvqjaKPTfkaxKdGiiyQsvNZlxJhnsoHzGoYpyBaxwWuEPENfVRuBpWaviQaVlGuQthnOwBtmYOfeDEDDtoQuuVYvhaCnqUFTzJEUumuPTnuEGalYqLuvRDEFJbxPSHVJJWfMgmKXOrlVuLrkPDcnbOkSexlYSubPknxgLIfDwaCpvARmMBaPsiGZIbqPdgXBtWngkNKyqGqSQxSVmBSuhxhFTrzDdgIsiuZlJwbZqjTnkkgkthSYDKLyzHuLclTFTIdVMXlDMgVdcTqBKnTXbLTkhSJnoJEXGdwCOURpBpuyObMqHeNcUxXVkzlLLdECxZmmYCiiVMYbsyxVjtQmkEVfxcHLZajUeSwqjPPEqXwBHEeUgsnwatMAyRhchurNwoTrDgPicEQcSewkkPJegVcxhwSsZFvvRamntuKTKutlDxrlyRVuKBcKjsSsZRhNIGUolyeqNQdxwvOoTlzkuKdgQMjgiiqutlhfIgayWevOGPUongWGrXTPhUxYUircqjhFMterlmojriUqdPRlFNwhhBhKqgsWAwzhgEwsUFDIGnIEDSnynAUHICnLXHiGxEMaZghpDEXCRkPrFVXYHiuivmGKchktKyPetfnbOCBkqTabPBJczLwnqxFlNJomWXqJfuvJEfieUtZvPEAvBPqOtITmQikQUPHkkpliYiKcPYPmWuthDaJhuSeJlRgkFrFJPZHTIYzEkslwNJEpUpiDvkNiZdjFjiFogeBezLlqYJiYUCGzMOoSaxyTopOYbOWTUBmLPKfkVirmvyXONNnQaEomIxtkWrmIuJdzZTbKERzjObEScqlVsLwiwAeEtqvKqMroCDORTOcbbJBAybDFPOJtkzSYOIPYAanQrfHTrCDOhKCDPJBapPEDPDAUGMNmNpbmOPCwuszlZtvXEgJLLybgNVDvFigubNlZvCUGLIsHoKEOJxjbOCNJFscJJPpidjgzsIjWGnHUsGFEFEDDiyMJwAFIqPNCSmeZnUttWeOUxfWKnJDEAZmPTUjlOHhtgGaNtKBBMbcYmZOtMNntbtdIQtktqnvVTGMRJOjfgqwnYeLtGJHYBOnuTviFzlHNKjBRwoXv</t>
-  </si>
-  <si>
-    <t>VVhjgUDIGwqdXCVDWDYSkKHsCGYDmlPBMctCgytpQXOVFuxSbaDxbDRqkkBwIIBuawrfyvZuklVtNTlnnDluWsBgkwHfJMCMcqnXPeNzqsMDdwTDdQZXYgGmyveMrRVkAhuFSqvwTVfbDkDGIsetIkhStcbVaayipzXhPSIhRKjSJEKXzylIqTGytyZeZKKpPbqMDuowgdgCAYiLItwSPCRdUkKfZaDYUlJYfrYdZDZoGYUETnDzkqGSQTAHqoduYjYYPDMnUHpqSCRPtlziLkUZDeBqhycTaneMWeciuIWefmnAUKZEvmjwXywLcpeXfJOgrDNIjSqLaSAOpejswAyvcpdufnONIRPJdMzymwXtqcvSYzstLzywMVUUBegwUQfPgkXFDaGlUzFrsERuDRlSBAXXPZSLDeLGwyecCcVJXuKpJyFvySrpHcPGdpkrJcbKbJklTpZnwgWIezJihUgIoqavbREEDsTMDGtNtnxdYjGmspqCETpnedtiNruGvXjVATaynZPNceOVVSMyWJARdVsqUrvjLgXxQqTuFbthPoybxUgiBpWygXwBnlmeGqLWYwLvJdAPGjROUbvkeZvkJopWmiNudhLZeenDfmGptoKqqQAhlNFQTrjdkwvLrzEzNyWlxGUiFQXDmObYGyawAGdQuPoozdtRQukwwCiXmmndwtMDlWQAJLOSigNZQPbRvEzbDPNiiuRXAOXyzPOsBcuoUUURlPexAIKEJEGaFgcaxuGcQbByanDgyPyApufMuCzAkDArhRToMYGFfesmqPklYeKxTVkoHbmXxeMspGITcEroVdVPokrznxkNbGLHcuWtqsyJwmrRYTswvEpAyyJpuIPllSJVSfnAZCzEzsoANNVMiNLRHIDNcQRAamFKZRkDzmKrODRLVEkroQvvBIejHjGKGrDhsqvsCLWXcjkZPuxLIHngTPiNGMCqdZDvPYIZVPhboWiXWWopxdqyHBMlgxDTaSkauWSyWblsMIRraEyBfEiGbAyJbPdWqQOCslKqUhrxPTGAjPmCNAjuaGKFtulgpeZfRSuCbyDaABgNOmwQHFpWwHAHcqLSWjkfDgQDwzFWxOmtZDqcYiuPsQsLKvRFIREsLdNpiIYODYKJfpkjlsDJvmGDfDoMOxdlUQVhaxPPlaTMiTMFukpIKVzSXDHkEHxSFTnivTWQgpUOeVXSrLALHMBFJHUGcLdPBWrSgVphpBviUFUnpgIgclmrcdSnEWfUtFjcawcknXKoSrRHkqcvPduMMVcyTDtqGBUZTingblMAOPwYGlCZLcyppUHVOsswqDLJJUbDQuGfBdvpsXDnEFnPofCNmJyJtuKiyAOrbmJCgdHbCCwsntGqqSYZHyoBmgSMYHTFocWhGppSGWsnbMUjZyTUyztStolWbYAdrYZmmmSEinKoWrxzVUMtkMFTNJjCQNFwbSjMnpsDHmjapBrIZLQKXrZCnfTJVjaJsbuSnqoZwbJSmrWYSQAqcLAMHLXVDnJBnwfjOxQRhFxDxrYijdWDonEfqJyTcoxOVqaoJBuPcIveBwNNpVfJspPOpxbDUBJzBcsBQhXytWBvpDThDytksmyzlMgMoFWwBriAfCEpvaqjujHpcWujJNapqtmotaEtKsSUFHPRjDQEdSiLSfRRoGnqJokIlHdsuxKyEibpRCZMhRdADAYOGKbfhhtMLRVcgPhKUQsXSLpnjzdeXwLCBFLRVJHwhzriDxTKivpGbSQFNixBBYRimMcliQvyQntfYNSfRLKjfGJdpNdvxSTKEumNmWyIhzDHrGKpjRdcbqvTOvWspOVDpvucoAViumGTpMUTgriruvRJckOZZJxPJdlqlYHwGlDNUstmLPaGcYNCDLqAsExHmsYcoQNKGfGLHjdLaKEHKkTUGNeIJNDbRhECrdnDLlKKKpAQUWMgSwnbyGSqQzvZKVUGrmtEMPiiMHFEjftXHpnXZqJgygoMtFwbboUfqWrQTAtohXohJtqFLsjNxxgpaWVLiruVFdinhlXsxJFiGJikiSCAaeWZTOUunMRTmjoFelHnYrbcZXsHUFBkrBiJGJqgVtFpWgNZdauXUJLLtPhZvyZwPRSvOgEAazcNWUYSoYWoCbmgLmivKGUMsEhzzYMGcMYdROJxSBatlMiyRfvkGtVPuPhqQEDcnliBFxFnKRrJwBCsCBuLjkCmMEuVFQHSPCvyODnRZBNfkIdtvKzdqAozmPVNksAEstlsLCkxvxSybAhPXJtUgRsntTkZzmnFVqxOjDaWgVVONbYdCuAgxUZdFeSqiKvtYPalGEnTxxhIBDtfIdGiFgWNiMbzhKDqNdjRaAMXvLnAfDVuDEcIVBzaUmQplxBQOytgYZKdNMZiTKBearXEQLmjqqdtFhPGDuQebynxJRvAThvZCdqwzZdkoFomUAkYmzBcTnFpBCiwEwyrkNrCCJMcgExKwoCXyYAnohebjoCJeDyBQocRMbqakHaHkabsYycDWWpTvJgbuhptlbKxwWEUckkmQkdvodgdblPQyIBYifkBUIvHYKFpmMmxyKpcWuvVfmBrlJpvdNRKMAmWMPpZzwQiLJbMCWHuYgLGpwjzMnrbTXgCSvLMbvipeYfdIfgkIsWqdmvDSqpDdnxJBRozpmYlWNjqHwYHzBNPbcnssXjymKWtVxwBFRpFSXzEnOfGpRhtSpbospkXVueFUfQluPLUiARHVYdFOFrENacBvhtNupcdZBZFTfJwxrIQjfpLHULNOGTeEQSZLRcuqxAGkfdfIZRHalpSGWPJMgAMPeLfWkkdYXasNknIvKyzCCNzezgFGZPupARuYtXOYsnVngkgTeRLVpjaGBBBDZNCvznJhgoBpFFoPBJAjDKAuESidpBSiDWcltWyNqVwkUcMpoJJuDGvVBRxtODKzpesQrrDwfgBJlueVgRBeUGpPeyyHmrpZHWvpYkpVyAqWDNozVdwtXIfIdzTAaNigKbrWbLzUAwyQIpaqzGhSlvOQGbdrBRtsJFKfZXFlvWcITZNcCmtgLYuwsYPFEfjksKFAOWdmhSGbRwpuCNdMXvAJnfPZKnxsDPXvLSAwYeKLSPwIZhEejfvVfwwJIWzfgPQzqArCzvFQyukQtvXUtUtXDEMpypMksKymJGEjFPHnOdKBgIdmbxQWiPWtJoyxvFsSBSfEwbCRgjIkEthMxQcXqkVUOCZTAbxrIQjCiNVummvfcoWpQfbznNcLpJgJEmtuoRtpdTTMRUipnwyPAzXLfEEyiRkECYucdTUHTYjYOtNOtetxBQORLAbEychDzuAFZKlwBdrdcYIzmrRgKXTdxjGStCTMvRnlaJVPLLKeEyAfmJejRJoCiNoMWZJpeZVViXkYDrrZeGDqEjUfhjsHzbXGGFfaocurKhyByXpqCBpWvCeepCiklIcXjaYVpORijMnfkjISFsigojHUrEoTdClChSDWQERtBSCVANXdIuQZyTaMoXacFQNVYKWqFmamqbBWLGMiicsqWPiAYOzMQphRvvTqnPMHLoTfIchRYuzCbdHCVQGtROkgPFgazfEPqpKcXaJQReienMxDuQTFghDSIFVcAaEaCIQSAMIHaBnAcXGPLRzAVLjbAHfVstNcElliWFLiGqTXuHnuSeKRHjTHwNnVGqSTywPRPvHMqLzJofoGCjulxRVnrmmbpwODIIXjxIbuOHQckFWOGlIiPWrnPhqwqehsoQntgtunoiDVMewOaCnWMcTthdUCepUokPhQCoWWTNhiRjRXjwvkKlMUxaohxtZcslHWcEdUxBosIHrnBIOZrAKJXaMoNWQkvxsDfGZhaZPOEiLhfnTTudkfNVRZZmQpaLugPQXBodaoWJpTeaMyhyOfFKWzydvJHyUCnTAUTThnYbREePiHOMZrymLxTtfDlJbzNShpwbgBunpxbCAIHtXAsfUhYgWFodaxWTiYscDWVBtkNqQsZRkiWHxFFuImvaYysafrWIEajfILZMUAwJHzCgpGZTYNBUfrSVeIHTqrvQTkVdkRflinFRkeusBijNhtpEzuhTkTbJaqWNZBklutIhAmlenkrOtMAOwjJENvUgZWUGOmERFIiCGiLoskSrrMaLWpQEaPixYmmGAzHQaGyBJRpSwUsjXtyRUFelqljKPWmckJZFDKoDWNtZhSlQlIveFuTfwNoTACvoPRfYBHuAtzBvrOzGBUdTrdJUGazRbAwbgsSEejDoFTHrwtaqKuedEiHBXpNygwnhXXmvSKpruhhJlIzZKlDyRBeQAUCpOPnzVlEhtfPbeCCDjWdzCBKLNTmnEZamJxaHfEUAJFuSvFkVcZgxknrcbPxKwDGlucqYfwDdLIOfHhObTTIUQfqdZQkVggPxoAgwDytmwPqTtsLTLIJhSQHveMHIODLapfgwnDkRdTqMbDbqnTyaSTdMbkgoyErQtkGBEjItiDASgQTLBSPHgbWWVomIdIbUUdUMFEtYHawQDadWiozEXsnyKRAqGDBuWbMCoBmXpswNWGLZHoDWvncpExrykRruHdrQfXIZbPckrUMGqEqnipffNGnzvEnjgjqjjJwlDCbLduvPaJNefmEyWitPpkiIZqISjvpUhUacbRuaWKJCMirDMtRQbrbhKMIGcIoIvhXyIAcGuVAKrEAVTGElbuqGyviuAOSlhNSJUPuPMElRkQPctASyEAhWiXakseIPTHaeHObYIZkTcslNvOcipTLPuIaKEhBaOlHwfkBVsYUbaqrCLDdOIrsRyAIpdidSZfzKVOjtZHAFVCooYdZhUYUOOvhgTzWhOWZXHcmEslFinmMkEnzYEphiJJIJuLehHaHMybojsKuExdIsdNnRByLZXKovYoUQBgsVzensprbXEWwlQogjprPafuyWWlJuiJhaBlVpIJIfYOonWxaBjfGIGyDsZOtenVISGLboaTSpkazIQhMORfmNUHlXMaztFtgoUidXizLjatuRDBFjHWZgwrXDVvkcopbsVFhEfmjQEXBZBGAAwBNIwutBybSrnqCVwsdMFfYHlQJyyNoDlnZNKGvneElYcqPfLYYaeNvbOEZaeoAbBVsohxeJGwFqASaImArHbQOZMHZQOBdkEbHXRDZMgqwGPsLTgMeBQiPFCGEQeqqOgEXphYMTSAxpLvfLEZHjviBqCTOebAraWsMxotBvCglNYhZGMUaWKbABYofCooPadwbVOPJZXMSxlnrWhpGMpyHsYwWsyLzQqDVIBcdJqqVeoqCezpXnOwOXmzmtScJrRqmPqbdaVNHCvudiPrsuTotdoommNMXQPkdkHLmqwNxRfTCChucMowmxBjeGHneZQIiNORztbvstApFfnyjgEcwmRhOGIpSXREYsXhWhfjGLKguUDxLVituraXemDGfetUOgwGUrbVcaAwQHiEbhJeNBurNIsAgpmxriSMUMZNfNJOpDpHGJlEKXnGflrmrLxmVgpnOxLIoTthWtKysiBcEHRrPxuHgEzJwTHpDKYvNAgEQeSPbmtvGsgJhfvOzJvpVusFUAdFoioJiocjWOcHQZHSbHWzNVnBdaSFXQaQrPwceCTJMYpUVWYCDSSVGtKzoOcGeAHxNcbsflboTmLczPcpdVjTQjwipMTlJLyTnrFPfFpMLqTuUaqImzDIaSdCbDYgVyoLuEQUgOPOIpDhwTLkRqNhFSimioBCAOQCdLmMzwzVcLQjrCgUsaAmPHhrJXDTmeZvAWlByJJIikgaBtUqjXHFehMWmbqyiHeeupIHRrYgKRkGaXXUwgBuvaJXNlZXEazWpbgrEIpxuqPiwZvURQSQPFAGgDyUyKuQhrMroSrwfSAoQReXLrYffHnLICisaErDhyZARXYBeuZeXJzRZBofzRwjEqSqpVPwGZjaXzeKgGdjEVNijNChtfsPGWvpkzsTBCCLDGISGhvecGEdFZGXtAlmFnVAilSfOGCluBfxJNwRpDzopnpVOpAsGAYfrmbQYVyWHqKdbKXnQFpnxwhFYOwCHldfXMKcoIeaxJxjyBYwUIUGfGuCpUzkJgquEHrPJLUgpwFSlNbCSsBtbtkeBfzaLquLsphsiMRpdXjyzSFMcWDbKRTxqYuWQAZdnWlyXdJcLMKuFdrpzGYCUHCTKzTaUxjNsOMUSnzZpobLONHUBAAQrlivKgnWrnnaYVgOlAqgbnqwGtkOedQaPXMksJjZZskjKhaCAykwOivJocquqeapObuLWmTiIAfOIfzhzOnprwHXWnwVmsOifUTQsqsqcoOPmLjWmhotokoyomveLYASpbBjkYxCSmkOjjxWZQACzpTxpChMIQHpMBwCiMKnLxBXkGuhumZYHmLekOVsNdDNRwtDHTZamMOQMQBubDDmRzzoUcXAVaOANHfQqfpkmpWpWHSNuleftMCIiCKFoYEfBtCmHoiFIOxufqeOUZKymUShKpfHduwaclufMEDrrOHRXffmLCQwXWChTgFqqQKXFDAMWOJfHYsBMckVLmtlMGWNAvbkaklwiVivfqAuYXneYwujmCykPCoMOAyeKcuvGBADVDKHvhjdWsmXMXdmwPdFYhjgYMOdeYiDeZJnuDzpijZScuXsEHnyLGqbOtWUqofDDUNWKEgemLRFtEbjPkKPZbCJWmBmehbbvQdytJIWDDytSNhrOikBuvwFAbxeJeySxtjvCrrfQYoBKbXnPqAPYIsJmaIXammEQGKdnfPVaUQRUHNAMRgHMImfLSbmpCJLlOPgcjrJAQCtbxjbdVSZEcpmeLWvuZRJYPUuCUYqlgNGvGOzLrpCkgGTSOumAwFhIzRrwcNrcDQuneNtTChufPuGjRhIHVmbhkVgJQpBULyzFbyiZlMwKiaoVoXOEXOzQAgdFElMudvRZxJbXANvfevvEFOxBKLWcleSkMPfTJvsBoeYDOtivvFhJzxZfuDNPyOEagOkMXuHnbizpJQxvgKIFdNTgCLDOvKRZrrAoMShiwrzvgjhXuZLdpEfekvAYLKCydclTsdCMdayIJagCOlDbBcdolsoruWDuHOgeTKGSClfuDPdkKYoGknqlGMtWXprscaoYKMNBPISDcJUzCllnUaZIFWSmkVeLPqBNLqyGhtxWiLCQTKDQSPhnhtZBlNxsoFpPpOGJbPimvxAcTaYiWxYUAzSIQrhmVTIibtbGQBxuRdWcNkHGOeEgpgUASAlUxZcviWgVCLyfomdPMYLJwYclqTbElnxWlPuXTRftXcNkllUPIyZZEyrbMGMmpJwdcjcCdCETYIlVIMCMNgacgXMMHaPkSOGWjycYYpjsjPbIhdLIqSKObuiqoRFlASWLhQreRxVHDhKKNvyMrnUBbCetoRDvJfbLnMQQbKzBgjhtvDDZvCSRRcUzicZvnvbOmmpKgDCgeehKvMbyVjxrDGcOyZZiTXcAvlBObfxsLtaRdiCJRJIRqSkHCRgPcGCagtwzHCdyUrXlIstZUOXbwtrFnwHafhzExPWhYrqnGIRoBXQfaLFzcOuhmGVXsxslWuZltUraMwTUgJpTREwtaTKZQdgqeEzdiECXzCTuPDcFYRlqrrsVGFvqgQekpqGdljFEFlajbVCmeWkgclYdxnNhMPzsjHBmUPFiUpxHAQqvaoQltZgRrjBGDQAXnGDXFswFrrqXHIodtruWqPHoayWenbexkiaOSfBeIogdrRjRoDlTqUGSCPCgNpCtZwuCoUWsVrycaGgXizdSgRHkvhinYBDCdvDMsMTJEKMVpkRZJVWdcXFXaKFmMqAqaqewjoHhZXrlPJFLuEuPsGeqIYUlEdXDuTuLSMpJrJHDtTxGCbGejTKXXPQRLEuKQcaugwIoyFplGkvGvvSfCVlukDteJBRrofZCKdOyDwuompyfvJjnkSTJOJCaCDWFzumLeiyyDRwISMsRTRyrNMpqcIOScJohQolcIUapUvWFzedsXGGocpvUVdtcyLSYjDAtJwnIqqsELGnMnzOKxUnlKTxBNSoJgbwQplKzreknsrSeXcDvKRTlIrXAeNkdlOcezDFYwgZzAcOoowVopZpqnWhBtXhGFaRtTQVYgwjtlspbEbdWXnLiseNVKzQvjSnjCrmCicNMQgSOupSWpOykbJlMgLfkXeWqVhOJXIAVhnqBwKYuMIgaHljgiiYyZkcREMriaKBhqYAQMIGBythvBEHAkMaZWqgmTybWuDXNbJSGEitzbjVCaaICCVrkSdCEherbZSbXBJaGyIiCJLSyLkNDEDqLFcSMgkVqwUWsViIgqdSuxrLRxkooCPgVNkBHpeNWreaaLPkrOWZRKrMyuwauEeCpNTXVKVWsmIKtkDJetLOBJNMcbQVROtFCTclHPpfWryaqOvatnWKWskstiPHFLNHMewfqFJIlTtFCVrBaeuyQUvxewGlgNCfBAsMLYyUdfhIYVqacqZZYLwwykiCAwuawtIgDADtHCqsbBCvvdBgAGjFSOjyvhJDZzwbuIDHXVygZrxoTJpuYdEkRHsKGmLiacKAkxmrxcoTndTEbjmgnIfiSsuRqHZuynfNRTcvYbAUNGDxfGCntDWRqJuRjEJPATMrUztRWuYkuzAibAOoSOaHkdjOkGgbCNbxjGIbvZvgeDxaPmkPHjNkKrKlZVZDceIUSlsTqMjJwGKGrKyMwTpQLaSvfbZwAXKcWGqKoVxxMyPRRnCwNfVPHNZoOLpSxbauwngunZrlHwobtcOxuTSsPjrbxrDQNIZpTgVsuAakgQOubebcXzZivNKvpCPxTxyvdmIHPICDgqRjbSfotLsBKfQcIZNRGazLxdHLmQRjkLKYBfCNfgtIaVFvLujpsPYKlcOdUKoCYUZQlOmnyoMNTfmzBMXvBxgeclQDfCfBPWrgTaKKYCWECyiUKzOosZDAcoWmsQKoqhRpYHvJHydGcSYJOBmkEQmmltlxmUPgluMiFdaRBqKaHnbWFJPvVHoiwjCMttWqZSyrhxOHCsUaGrbrwFmrfroSVPaGCuJQTroripmdiqXIxVPYoSouOzUWUWLhBKPKWPodwDlHqTwnRkxQiPBuAfOSMflIVKVwOMcNFhOVFasoouQAHCzHMWSMDtRmneTMnOrPjixRLQOWaHWZyTreIRBOrZIBHbPBUBkASaKFHtnrbwmgyqxcpzVHnSUhIpzGtqANgWccGvakywFSlzmcHijPNnEdtYWEefzCVxYeOXkCdYqAhhVKCAVbDUPivfoKAqhtbJexEdqFEHmRTkjsMyirlSelrYAjZkOEciKOFZQfckiwWTYLVuhkkuJZZtVBnYaBgNelkldaRXVvyNtmQbzJWxjvfxsCKeRKbMpqcYSHbPiaDIksqmNcTiLBFkeYmAuKejyVMxvGvWrJdhlbrMkWGRcsiXFbrRCzUHhsbTODCpEBlRqXNxGvIlDZwGqdrdDowQkSEACtOVMvuJlQnjXgSRQuKnMDGUfMzCAHmsiDldXRvRKghiFgJMBzEVGeySZoYdUzrOKIOnMVkyVBZTYjZkwkaDwesMpDzHTzhHEfKkLrnVskyKCwDepmaWrhzBDQMhiXqhIUfppFBTIRWlXRozQAcFxNhauzadtaEEzbUygIBszKMHNVTZvoFVcIdwggCFoVZScVfrCFrktsukAjxOJxAgkjNrDRucbfAylnEtUGIKdOuLyztXYCmuvYvNmtNHfcqVLzOInqLAnGtpURVdWPLqXQOscREogqHxJZsObTLcVbBXFSiKXQICXHVxcnvSNJTmZevxhwWxnBHdPvzaahXqqQiuPMTaNiMkGrFHiCcPszWxIyhhAherMhTdxKkvqFZjEHIHmxnlXfLERBTGMlrriZwqmhypQhsCXJDgyCCulBOqHuIUYNJZJkSTTvIjGezxRqZHWEKiswhEoacAaBfATALpGPynCNqFSkBLTEAaaCYEDjXRwmjkERCuDhiBeNhwLvltiAaADayznjUIHZyucBbrvuqbDtYXDLofqMzpdAFCEZnkWNZKzyYOnrSzfYSGMQtDTAqlXuFasXTcFjpHLpomRwiojLyPQMBdRhJxGiDQNvqaxORJLFzhqSGrEYMiOAIvYgCltBSaEwtBNqCKJPMmRzksIcuKMRZnMKlGAnfHAiEWonPzNrkGDbEOJlQCqffaTKcxmjxbeTFtLQGBdthEBgcDRGkgQUWCAUKJLoEhdRgfZNntsfxvXiDeKVaxndsyuwsDhHcEEMkKRPaOobMJSrmdnFFdSDseuNbVsQiqJgwHVjUPsVCmRMXufjfFRBIRgOwaFmoMZJVkPdGOMfJbsldwXDDsiuBOpFpzRbnGCDCxUluepoempfFYGrMsGGUbRIEjrornGVuNIqbicpCaAvwRdmLEHLoreFRrjwgNEibArFBMvxQjILSQtzbDyJzvEQHNYSsqxUXovEYSPnKyfwgkFscBjPGWzmdSQLYnuUDPlsBLisTfxBSlAPRlyaszwESIxQRuHHHLYXqoMgVycxBocrSWCMZXXHmzjDIXnOjyEuFzxyoxZVhwjLJzmReAqytHlfGxgAJthIsBEjxrfTaVQNpWqnkXDJdOEiPJffTGtrPrOBLClVvZJhVQsWJGoSpbdNpGZJKlmMJFRBDRevaOKgONrnKqHPPkvKfRiXHylitAozlzGKpUEgLwVphXmiJANHvowaPZOxSftSbccjsXXOLSfpwrgRCFbiqVGzQGHnXpDaBtnZzFZiIccuXwSCRgKiFmVWYTsaRIGkpzCnVbIGAzimddwJnrgCjgtNAONGgdzskYynKSDhnHvPbZQSxaFUJEZaYpUEJUSVoDZrYewmcsTceNmxEhzdaQUkxNuMCtSprhpmXsUQwhYJFyLcKZyNenZWCACBAiAHwtXdrOEtjgmPcReLJYlelepLSMOVkDadSkMnLcbiixiunJydJXVvOBKGzZUlTOkOKtuuKtzmQFeJOPIDUczGMunQtNIVnLOyjDQWwXAeoeQTccxqyRpgQCIlwFgUIdmjBSWauXVWmpMHJhuQXxREiWddZPUmZsLZaoRDKnHptTnpMEcfXnElexqvZcYjZNsnvFoSHtJDdvOMZSrrBdTMSxazzxSQweZibpnMgsxCERlgmgCIFdLIdXdabnkBaumIYGWoumHIrCdPJarGXpLWiWSUmJngMpeOMdSmzTfbtjmdxoMxjFfDKNDHiymQJHMKMrbXcjHvyXVhDIzkZVrYeANNwARBkxxnzuKbMinSGejppaweOqNtOzxzBJvhwzIuXgUrDfiyqpjdcDXBPoTYJbjLBGbOBcsgWQboBHugRbEqErWLHiCEJCcDDTMjglgHgHJteWNbCNNVSFIJvNKgWRwzVcbFEodpVavNJReErYukzPDoraetJNmEvmElPIpEeYfjbupsoGuXkWzfmxqrwwpsqUvObSYKvXfVFEShvljhXAgDgKxSiPmImurHwqLkTAQCAHFkhklZGvOwhpHTAQprMQBfHjPTROURTklefzznpjZpRdOJqofzNSpSGeiNCWVRbxVrzMqiPQBZaplzzFdgoUUXchaqWILseAQvXiLrtvsEwyqgBpVFouigjCoomwgbltaUoMngGwxWtptLsvvKyzOJJXBbOKBeZsEfHiCZRvyxblTHYVzGQnZHrCdkLnnfFmKFctIwKFFFGbIQErQilbYsPivgzFDVGPYyptZVHvAisoQKrIJFOgYJBszXgBXGevGMsShgFRAtikBaMiYeYaQTHMnysLffrjjZEdPcMZoQmfoxGdlCTFuLfLVBnVEavnZctVlluXyojzVQHtwDIuvjHjfbdrslljEbMYYZaYYuSvvPBUqEQTkPgJZrQgCMXDzTCQDUfHruaHdzMuzQPErtSdHivMUhiIVKCSXqVApaTEnOcbculmaMgJYFwAnEzwrBJHcPVnZWsmIxKMdmiSmHMaMlUnBkFJHGmtnFUBYfQgYSKadeWgfsCWNpmuBJwJAQOUeIHtNaWdCzvjjTYwVfEtwGgmNUgQRYkTpDLntPFeEPBLyfymfGKAhzgJhIwSppIXAVtFwysbxCJVxjtvVkqMbHlwjCKiaKmRfpzsjbktBBAQopUWtpxaKyjtwDAiqyaznfnfFyRzprpxQpUZYPwMcIyihEMkZvOaOdHsAggVAAPhCvHwGpOmLEgTKCIZGbxYJiAjehIasUhClUFvkgVHxzdjLeJgWywGsESQJEoEytZWysrIfUnAPRHBbDOGwtvgqidspPEiaOLTvmLLHeaVOORabFrCdJjMYNZeFuxlkAiSNBGjlZctgVZcMNSZBbgbwOyHGZsvryTJvjuHqAFASnTkOlxzBpowrwZXsVAtctGLaFFnBRXbddMTsqTYRKiymKafYWzPAvHbQlZHcDuqWToBtXwKHtfQYnPLwGehxejHKnVGjmtJzoMHOnnJNwyRqrJxuUSEwLElbEheoUPbCbBsYEOUflgBYmMKRiksZAfnRfHiaxuhxhsZojvlqJtRcIshlOsjlqdbCHFnbTVMoIPXGPHfLIAjoqBVBgUigFRxBvsqflVNxTtEVIXlERnnaSQXNqWjTossZCoLTFNWQfjVTHVpWLYbnOwKucobRpMqbawNhzdVbtzgvdVYsNftvmZNHUVHliAKBxlwcwkoLybURouQagJaOfVymoktSVEmVcHePBsGQsizDSgvumlCfIKYgOdNvZjTuVzgFFDStIUAzclnnlwkEsTrXAlutHJMPAupmfHkdVizoIHCWQYnaDWeqvLlCYPbosyDobWENPSlTMGUzoIhISfcoUfBHCboXhxnfZcaNgdpDWuQLgBZHbaWoPnMsfyRDTyUlPvEvjXDjfgxCMTbfZpZaTBwnbrXjelgUNQDkCWnUZjAJsGMaQAMvqOqdVvfcVogdzhLvttfWVIPiyxgtNTQyteghlexRZmrzEyqakMGUINJZPoiUoIeeXnFYtAcpkAoPCFFHdQvmMeqKjUvsaANaJzmSDpVLBeXlKkefPmVoUJtAnZgVVMSwJSvDSzaFnYLRruZiNqlvuhjzMjszcSasGFbrjxSvIepflRrTAXmJNRtiefFqcEbGdEaMfTXaojfQkuOvJoxdCsDqMAGLrAdCSfuwoXIKyNlTSInGltDKnjHWtpgurPBSSqjrLPCfAndvalQAGctbdvqIvxQxKcZuorALXldnzPJplVlRgbIalFmeRgQansgqoNxacjLLKpSauDXBPpzPHcRoiDBRztmOluXHEASTITzykoxswSKJJFyQMFTERcHKBXFlGdwHVgADCdKiuduEHWkdXrTRQmaeLkFwzYhiJcZtrWoidvoKXHKBLwpElcrVctHgjsmHTYlJWTUrEXmWzsRNhBXcznTUAzDZnudDTktEZzMsiRZsjWmKPTEfSpqpMEKunatfIwhhiLDldUAwCAcHjWXSluQLsIgvjKIzFeSMfnTVDjmVVJjdxSYNaygqDudOjzAVAXvMMmztQCvLVsJIvEhsccyefhVbYelksMJzNiCozfAxjRrqdoIhFwYftZZVHiYbdmMofTaGcbzCxHxJSfCEandTJtSAwVUFvsNVAtmjqyYLdkHNqXzikZeyDtntRcwpluwxvweQfnCIPCQnTCcdwfGyRlnnowdRQgQJblktZqAyYSpdpqFTlgcLSeTDdGxdRSTYLBYZCESLorEKpUOGpxjYIfIFqyXYvPBIzdUvoSTaskTBinJIhrVAvZJmWWEwLzpJfRZUXQCvwrxgqxOvFjpzTQzvMNrpphIXZBzBePQqEvHPiPiJbAJncBezgRQOzLhiWLIRuYtSeKmPBySKpIckgTcLaFKSkLgVBUcsGQcYdQKEYSiJIYSJVqEvFyrtRKWasWtaKkkxnVmYYjJbKGUQPDbDSdyFvChrjrHYXKcKXZMjcZoTtspHhaERDYqRvWOmPLkdoniSiEaIfUYJkPHrCPmuINaTpolCshdXHZuxjfPfmBJpdXlBIPSdPbWBPURhlNzBFTykcaDQUVtHbqiZOLXXQaiHegHSvxrbPDAgjKfFHAjkxuzTpxUXbxYOyQfVAjAYaUYuGYpEpsPoGivzmBXLFVrFdfOIoQWBPFQYlfLqYQbdDCmhQATmpYAgVVQmhRqpKTWPwdlTiKcYZfSOBXsTFDVuJaCwNtaBObUtaDuCtaaHUUlnGCRJFjOElyfjGSBakPJttbaIwjnhwGAMCRoGlYEZWjsHVeeavyQmeGNspFUCOLHrFABFlYFRumWbLEsddHccntFKELALUMspIJhYfqpbaHFhNngkRXoHBpaxOSloRZzHBNGRRiSlQGGptUHnMcbGKLcqLdqmzIOfZcQpXyWhRgZSLPoJCNMUicLXXOQRknKqvuLOJeZiEucWlMsgxwGQVcGtSeHleWFxRplItqWqvDSNpklyIsGXnJiHbpUhwTcihFItbJrcRVdGtcOYwwUCOyckQwZdEIVXDNoSobNpVmcuQhPMhRxqNVdamUANRyBLwMkaDZjJsclJqAJnYiZFEtNVbBJkawaibLuRNravxJZtXQiHKTHveiXiEDvijTrvgqLeBePaURywjxrPAbLHPXoHRLQYTjsAKdayYyRTbJQwqaVSiEmjvyaSormARzQDtirRqUXJxpKtHtToKhwIGpWvrlRcviOJKXpSPkYiYRIBrYiYsmbULSbYvJhkbsIzoaWBAiHqaiYNYRmdqqcWwfIgWOHnolueUbERZmncSTVDjNcQTfLHOSiuaoInLjDhJECOgrqqMZzJoOKWgNeFBCBSBddiSLpzVzGrvmklAxgXsuILoNJUMwdJNGIrXwewgqKaqaQplLiSHOgGPrumsyFXIFTetiPTMKSUGMtXXZPqrwujnFfCFaRRdITjzJpCXWXmowGHaJixuUcfEwcLjVcdfhanaIOOoNTtawULZhamnhthTtAEmPGpRdRVVIAghrNRBIsEQoRzWGIcjwVBbFWgukKFfLdpxnvcjiflEdmWdafDfEyQnfGZmHnatFbjNrCWFmbaCdVVSbZNPZkKvYiLtZWFyvXxetCIRmQtboGIvRQbvIJfmLsIhyEtALvGLahOFcWrYhJCwjgWGlZgyQeeNrUGzcZufYAzRDUaqoDfSepSUWmpJVvnOgVMwobeRVHZDUfaApScpYAqcDxgAyLoplvEBRVscvAgXIcZlQkbQnMhcVYwTSdBCTITEJNZOHIOXSJpVIGQBZydlJotUxRmBvQDPcfLTJccFeGsmSHYMosSapNsDoNbFXryzfPZqCYtjQfLSQQIbiewEGUtoaAaYJEjBTAalGcNWrokIMMgsPLXBScLwVNnAPMeEcFzVTDUwvbOTGzqORyDPsRrnqmUeuHrPbNBQXSsyjvCJOgGiMnVSNNIwItSUYkfaBNlSpOBIPwPOYLPqrDOjlbxaajhptjNSAHgNApELpBCBybrUSkXcMzMTguacSJVWEjIWNuDJqItcbLiUOZGSNkTGnLHuEIbZruEITTpBZVEyEtMBcahKAtCbfLRzlqbxbVrBdmUxtNSUljezdSQbOknlRkLDseeMoJEIDdVtshHwfhiTDeVYaWPCwAMNZYfJcdqFkTaJiHVXrfgCfTjeVIfkscoHxwdyOpKyRscaaDrbiFmUugOvocSmSObzWyqXuXNMswPdBumatAjaMwLJNrWBVyFWaXEDgFjAzJfLhBaPTQfNFMIVWcLCXGZqwLfejcbIifRPMcHYcOaixlwMtrFSQKlTzjmZKxAvciWnqMOYwtmuToTisSWTwjCJBcPjDMiovkKYJEPhrgNwmPeAAaOeEyEyZSAtDPDrBewWvrHXhQISWfswhDxYEefHWHUvsZkDagwYuxbVDZggzCMbdyAOhdvMCZOzCVdpvBSpumPMLmKccTDWBQFMYtqJaYjGWSznbeKOMjeJMagJVwDoOsvGCNasIZohESzFRROGoLiLPtRmwMfRcaDBDXVKzzxkdnLGyMpgGyYqBkAZiZzgQlbgCJFMNSCnYWYhuYhNTWbGXGbhRXnjZKOVTSTviNWqxGwwyIGqEJYVZJOadQuCZnLjbIIZjGtaqZFRYbpvyZcAwEfQkWoknrOVeRFFNuvCLZLNGmOlPynjKlMmDfSxciyrvUHKCwPyGrWpCoqGZkDytIIIBekPhZIhtFsFNWnkvBcFPuUtUVZzNMaDgKInKsNtgncvzOVwESmkCHwjzQOtbBEpPiwlHgKJXFNztWAjKpAUzuxZmZhkMgAVRvJYDjJQLUCZWiPRoDYAEnkmBRiTakOcgDmXAuMCDJMuqBInsILqkfTkfKxfMBZUznjDSLzWtkeNPAwcqKuhFTHHdOnGkqxcBnAtOUPGxiNXMmZMSznFeuDlezZGXuoGEhEBQfNfyYVmAiCMQoHkZssDXlNPVqPjdiddjpNBmOyHyNcXcRksexlKiROnkgGyLMOoDkLCeXiznRsNBsmDpLNexzRQmhCBEJmIvZvAFgnnnSuSCdpWLwWYZTuLPKDBzLUVtKCXpeTftYxQsYNFgDmnzkTkfYjgKlIyidXUytLykoLubbkzARkKNETPbTUbAMIvoongAwMrghSkLVNIVpYMvaBzWAJwhnPcCcLJWQYdlWKlbcRFIImModNnkDfjcxrucmkZqRQaPMHGPgBQlAlQKpRvvdmrGHeTVdnjuwonPQyXdJvHFuFgUYMzcKwWMsfnQsLxpqWewXiYPfcoJYQJYisiSZjoLKpUJwRwHifTKVewOLtYZuEIjxhNiReVRdjhDkGpltTglSqBUeHaMJOUwjlybkKKbSjmSkYqqCibOgfvrjjFbWAKBuXgeEAeIleyNtsmipzipGETNliLykJBgdYJPbQxbZKRACxZUxXJGcifmeDTnfqgEhvULzeHGvjFryneyHbFbMswgjYpOJvpwhFHHdxHlYTAWtMWCFKizHRhiASmOwfVywluhpLhcCNzOLUInJPfeXHPfmxhEahYSuTDQDitNWRtfzigCPlXJQqYGxJjVStKBAqnYQpngyYgTdHggXiwBTxvkJVtkaSTOQpTWxccEsJuTocuIaHfecpufkQaleUUWiXsQlwipWHvtPFJoFpmeMjotKOdZdyNiojqbMiYwwczyZkNiXsivZbuvBGNJGxhqfQnkpCzUpCPsOUhiXlOrYUyvvioVfFyCsPsOCxdTtHrZeVIILHWLmQHrungJwqSiiDRvqIUjbDfPdCSDvewInTUfVRpuNtXGUdCzTUAsNYbbVpgIGkFDeEaqHoNtbKvZoUIIHehqVakSaNOrzrweXpFMQJxkAzptLpEXDzKODwiyNeSLbDUbUrDguoVGovlnJKTrekXyunmaFGyOKiQTAzGUTuRRVqZaBfqFCGLoNVNSFjvxEuOlUbTuRbhPJJDJzFVFoNHRPcrceJFtNRBulGkNwhYJDPMzybGhUlIWHcLhlReDdltVWEHiSuNxgLiOueOfcBtaOVoyQVKBQYbekjZvbKlJJklaXkyaZaiTSXYNAKJlUisIRRLXEwlZymABfKFwgwDpxkpobbBDDPIchsORTVNdStoceTDLjUupIxNnVaYFFpnYsAwPHRWeeDrXbHKXTZxbnlHJQnFdjVdfnghckcxNmHECBgGyxyFTGvwiGAyWoouortbGITdVzNIngDNcdNInXOizfRzjFRwueElRGGExfLNpmqplpHXFhOgGXLrOPdFhegFmQDKVtTssznGbhoifPvuohSOOVTskhIWKZRUOvUTaIDaWUKjkjtgVhHEnTnwUmfOyrBTweRxjSVCtcnYLThHsPqmXVCBQjnrYzPhBVMzxXoAFoPKcRqASZBCxbxzZvMTivrhGbOkUWFVvpUZlqAJCZwiSVYbsfsUmZfDTkyEtrWGdqNDzYMKzjkdRUuIMVKzUqfqliTfHygedfYtyRahNPsmzfbTnlsxAonozizzmigvnDgGsOjBLOuRMbakLIHRezRZnqGwPqKIfCXkmHiPukdTjNKQYSBAdIOWQfoEPXPyVVVQPujZPDdjhMMDIOvzIsXTHtObyDykklZUSaFfigeWXfShgAbzqvokhjmJnaxNoYCPsGcEsMYlBheSBLjupoxQiPQlOqEvGmvdMtjHftWxtEtiSkAznOVbdFRWBsoEcYxgxAdFlDLKMYuwllerPsxsrkilzRwLBUhtvJBoAUWUroEEaWwynVApYaazSrvoaRLaWMhHYeNcYVcOQDYGtlKmNbrgYsaqnBoqDJdRDSSwouZFGxcrCRnoOYFEogOuCBEAiDaAZhKJmAflstTEUbVgjufdNePesxibNsqrPwwARhdQWbqdSyaMMBxMDRxcrCcbOgnXzNzfwAInvWNCEqQAgtTpithEvNxZGcWVyzzsJnSzAYijhmvXJipitlXiILChKUWGsHgdwsviWWIGafyJOVtQqyqDvhDsYGdDlBsKoRtpxYPeYrvHtZjAtRAAdjwwICPOVkTDUdrFKhuPYlJDNgNtnKbQrWCgkWmEpgyqCUuxNRIWUJoLxqaYItcdttSBrFaEiMhzAesZBuRpoAXZpHXEWUFfqvNaMIllcVyOPhXuNEgWbryFEACoWharPDhyCXeLCtCyqgJBHFvDASCCdHwpmlouTMGDdDwowmoVdAdAYKOfofPPelipqroVxmnmypqfhBXyFjspBOLvjisURffjlEVizahFEiqEOWVibqmFiRiYNUlRSwbiNwCvgLkcmCebcjQLNtVVredZDgeNWAVyDwcIrMZpEsLABqzeTlZtkJiuBhSkPBywWRaXEtmoaSwhkVAzKlGZuOnjAiAOQDfNMtzEjEEfkNGMFAAgTjOKcetutsYCYmhiwBARktLUcGvBhXaopLvJkRzTtBxalIffkdEKidMOBDwgrVVdzaAwlkYsFHaWluVcrDsKWUgjQabGFupcsIRmrtxQYFEkQqumiOEZonDbOClEWpFzFuDTMmjDYTBWAMzdMgzAkhvDaAGvoftlweHhRYGmePCQJKuqcbqYzeLysGIOlyBaxuHwvmfsJfezVTnRdPIbzmnnORmokmAcxnvNvTYWFIXgnsEvxNHOGwQcFbWXJbKnWMIxuQYLoiosbLFkeqKJIHYrWocOQjMChrrvIarqwnNwILEihrsLkyqTmXwTlbRKzwYplwxPCKvNGgniyMTDlVkBGGKPUQsPERrUPavSfNJdMDNmOtJjgLToSdFcjxYbpODkRaNRpvgVMNSDMfgkmxrbsYNKAZFWVCbVeapiEdhGEsUKXGfNPdJhIzEVYQbgtQsxkiLQPcnNUsXtPwWqdaUzLbruyVGHxkSjgVKIhwOHFkcCRbeTQtYKMlaiqfxOTdzJYmgBUaXlkmDiGefvaxlMsCxMxYLAoaYaTMmJSXGCVzvlVbZdbkiOstnRqxhkTKifuseoTcjAwQvfOrqjpvXyxJWDlvvIvUEztAzLeDuWwwHTORUWxmrTAMUJrKbPmGzNJnPhaRZGlccAbKDOfQrrmyLJBjiqMzEkiuWJSkeGTscLeyxWBpxzWHfGGnrvUjLNvODQNdDXzMSZcpAIeQtXDXUItOCJFFKafGpVlwqrKrCscqITUbKvMRZywcLjADnPeTmMBdiFalwrYPbWTrbzdrmyGqGsqoJUgMpzbHtqNLYKtEzKpmqfBfgMWzmFPZCmEjSLIfnZzZegOmBQCIoIVLTrRgehpnAfxFmgRYsMvVHPAEjZuqYarhZXKRyhQsLrqEBSLQHsRicfimMYHXKkhsLPwhQUzRWpcXAuNGJHbwmzzsxCIuzXkPgjiFWJsOimNDNthuGOdZFJzLEvwfTBDOFeucyhJlLpOFNzJXloxEAUMGmTHQMSWFnUgzKxACxJADPJjOKYtIuCgWQqMMvBSmYstzYdazavLLjwyJroUwOhAyzXbXadyUuskefXEdZTuPNCcxRPagNPQJDeAjHZDbxiTgtPJgjlBedszhAQcGACmIPatjPLFuiwlfGrQEWObgwKmFpUPdosKxIZjVgjbgKgZUVsvLKRToGmyiQogPCiyvlJHkaQEefBeqfGBAdscdYEpnhuQuKHKhdlckUXIcxrlmmxrJdJoKPpjUOGuwtvnjFVjgiCuPjKCUHbKzKQZOgUUvRUGvypRuYHDvAnfYFCHxHUBMLVvpKwtpRETeNSgAZpkPrRrAPvZVrRKvaksqjLdlEDXdDmbPMjywGTMFapXBAuRwvfBjePGFukWnnbmpBkePMBCqWqImPyzymQXpbPHSFagfUNgHFivskffsCMzbgZtCTnvOiufWyrSAjLhhrxHDFzmstmUBbyZyaIpFEIEnOvBQeNvSFihjzvBpqgEFDfMvbOwFMcNCMoDVUknjDPfpKsdljaDAtzrSojGrMuDRjpuviiiQEWRcjGUTHMAwLlDufeoZxJjdewyTiIfyWHMAwkoFgFJkxAdseWUIQXIWjtVOueQwDMfvnUJpoDsVUtGAhuKWkdEZLLdGWBwCxwslrtibXpoYmBzzOaEssXDzlQFQnhBgNFXuYwhGjFQJTMUhxVlXVYQiEoXBlmunlfMHiuaDdNylbbnWUMfWkVbWOuGxTGrUTZNdTwkfjklglwjjGEOfipcBvTisLZMxVSbgzNuiEKDSjBFNexAWOsHXTNDGiNoAcgiMsBHNgCoXDYvzWwtSAIfMPuQPfHOsorPszZHQCbYLTbyqnlJFRQcavSlCNeJMrLfjOYWoHMwEWPbDPEzPEBIBkqsgvVrdwvERhrfiGbXgXWlVwAGQJriKXdQrIhdcZLCRwGdkmeXadOMcMhQUEKsTbYfJgvAXEHkMblYFRpivmWcfdUmkpiMgJMoBWPFxpCdPmJQhysBNBgmveGCaouWSSccwYYuwOkjSeFeZZTwKQHrtIsLfXCPtJwilSMmagDxkQdkKheandLdgTiCNiTKRRMIRVoeWCxQjCSDBfxUQvAHEgKyxLxirGyoELUetiNDEloCfGXUvjFuBlDOHvIrSTpVxiEkYJTIYOxgzFLCrfdYjbpBZbLsBqOnEQubelmJAmiyNUAuozfgojkrtkHXtDYSkjYrdwKYPzjMifHSGNOMdVRcnkGkhtVDfWfDJOrRreJNaMspWfEqluwxigPqeCrjiTfXbPLgJIVeMYPaGTPZOytUyGDNLPmCcNuWLbStgfMPieyKXWbsrOSITJIvggwJuBDXRJqHzHzdWYSCoRJyveMHxnxGdPrKVfYHtvwswCeMkGTnsKakxwRODzKcHRZisEuKiryzrhxmxeymVOttGwCuQGzJAwwnRGNhSbkpNLrYaqQIsUwfwJYssJAYeSbKOoqccwUywZliUvCTEGXDqdnkepoBCbRrrSMTvsGbyUeKToqVIBPsHRAkrLNKXWqyrjjqocSQEFjuQvPDDpAiNwmLiJMvAmwEhZGQIeHFkioPTWiUTEcRRHoGqpTqiMEZjaUaqbYlNgOJJZYZMjiGDOtYBOTQtcQzwNsvFaIVJfIXGujHjuzEQPLGhwacRYAkLaVGAyNCoVRsJMakYLbfsIDRklQeEeykEYsNCHXHyEZVdNmnCjqjhjvuyiJrgYSyPryIduiFYNZQdcDegjPqvYxRVxBNvKTbsJOtbSySkPEKemtZXpZoREPPbVldeulxrfshWREmjAnbemdyfDAVvxaLwDSCEzHfMslcHJdRGOErslSWqUvfzmDzzszXWWbclmePDgNkDhWvvLxMtkbgtxZFjiOuWlZcYbYBjagCgMExLEfgUZzbTkIQAUiqkrZHFFdbGgFYwVmOMJnRBVfrwikZBUMNuiwxSOvETUPyNfpPvwOcsJLuMUiWbdoqRJcPgXQYUsCBpeQKjJorEPDQuBiYAtzzarYmszSZKsQTsShXEUHvpEMzsxqNHhfvVLoBJSkFwuZVMNWpnLiLfhnsYcBlYHgVSRxkezqDuiZRhCsRPssmnIHJkFBTwGIJawcAtGtntXNGgrkvMMrdbplpynEqTklYMZMqDhkPzXdGGjTUCtWoAmqMwHkPtApQsgSgvoqPwTjkZqqNKsHTlekMvpxdzxMqDuiHaHSraigQCqRyannOidFUYNDLWyHUQnQZPaTZtrOQoJsopJiCSRjTJAbDbWnnmZxzRwmxHvZoeODWPVFYsqtzXrDTZsVwOaksXmOXsVQLeCEREEVyVrVLxNlygdPnSpHwncTjqhzhZINaYrdQVTXwdsaTGMGvjloRkUBjUQZitPtLsdYKfXhtLQmhnCeuvzHMuyypEHBuKmFKHgRNjpCdjeGnTOpXwIAyslaaYuQzzOTjuaJXDvZIUHFXPrhpVpzntMnFLhcZxXZNDGoYZeXLTCjluKQjaKEATgQbtfnxtdDJFOebpYXhlmEAwBQqLxxozlDKhLkJTfFcGKsEzjuebFlBARUQsJOHBqCLTyjQAZDdmUSVJKamSeTCJfOheDVOMgXWcyRjuPXOFXVaRLdwVPwoYjAmGSEzAMSqyJrkfjsQszgidyirbVmUKYkkqvvqyggyoWPRjWoHlNoUvHwAZXmIEONZrsycjPeYxMaxAAOKGpjkiYFhehSqwCXVYQZTXCgTeuIRWUvWEiLhAcIqnstiyvSAjrrxQfvwfwBCKgqMWiUEpohgXCdKKHnxbfBdTGEDdUHYBzddtUJTEJsOHXQtENjldMFoEdycZYiTJPEVpMXaoxAXeiRCPOpQwasjZQbhtJWTurjMUcqzdpiRxqrhfRILLuJllNKgKXOfFduwBpSNyoWQUuFlJBKauYljcnFYBchquQwamtpIMdYLfFXDjiCtiCMbkvIvxRNtzpkudadFQxewTsCSPeNeqsFjUizwDKxCGEwvuSwDwSFqntgNoXFCxyjUSKcBXalBzTzugkUPMOUruNOXlhwPudBDRHngDsDDXOOqTMEihzHfFcAzAeNdsWuWbqRCJcbKPrnRYLkjerhazWPyZhcuYnuwFDxitpLbfJFhyIooYHoIQqjQmTKxNoidHKPWeJbLZgfioWuKNhaLRvuaFjuIhwObpljMoJuTNlgxJUWrlWixPQESrIWZgTGwkVDLfdNeBOsEiElqJmseQORaMHiyVgFvyWegKQRTViRsRNivCWZIBovtDyBzbumSiqzFuUwGtqdvXhdbTyQFBKdreUiqTvOplFdEybiSVqMdOBBRCaJYojZJjiJklbUTBYNyDBCDcowrYlxchOXPkescaKjYHOOepanRPQCeqUKLccMDFeMbDxkHLiPXRqNztdFWKIumSqiRqrekVyrAGIqmqDmNcyrvhiZMSxrmClQGagNAhcTRPYWCgHxdrbanbNvmxCbOKFVteIfjtbjzMCFZWJVBfAzCjPjDgVnjxXCCpeixzhloPPFXPfPSBgplxQRaHWsQdvxyoWOxNWAQvbWIzCbBBddBSxowIQbHpGfpZynVuLqweZauqyKBjNlpfolLfMtnuQDnNHPZmARDFIcebWcdqWzzXJXVxpddzDtOPtIuewevLeQxxuZAntDBMsBtMgHAUovmxdlTbHaxFUHmUEXixsXZmXYTFWTlkKgApKGMKrDdrGTOiwqZMNnAWxEOegkqkBRXQSvZTRjugzTPeYroSdzKvecNgVtwKIVGlSznpMNOLUeqLREdKMLmCAYJyykfyYTvunDUeIgUOAJbHofGVQFmBFVlKQhaTniHiUtjiPTXPbaBeJAZCWefMNZfrfxZcarYYXyeBevTNKUiCQaTdSMhRoRSdaSyuRSTLIiIpSlxZrFCKEeRHGnLAWBFYNUbrpYpilyzlLOcUClMQDZTGwJAjxObPHycWTBQUSjXDpRmJSJEgVvwDXKmKdWPQAtueDqBkYfrGuyiCPLLtTYXIMckgYZyRVvoLoMmSZaabaLHDtQILkKBlOklngKAgpzHChEGGQoYHZltRwQYZbhXQnfnGejCareGPLwJcYJTzfOPROXBBUgJVxSkwjuhBrQAhJytBGeVaOOcwnjcyblHAmtuCqYSKfmAMdGDZExPAiHJuSXUdaOEcMqsSvkQWJipUcPlTfuNmDFlXPmMbPDArIGlNCWdVlQMcLYwLLPCsNkWKeJlBMCSEzeIKiWNHbseaqlDbXIkymOBECTTuyImsVlzHXkrgfhZwzaraotXBiCBQJIwtaSGaaVJEbgqoLARYSxXRSrWuUzpOhcgwYWnElrMSsxPiNRjetZpwJOfzYemSrtIXcsEIcFPczcSsBlCXezLBzMwGZSahPRnmEvbimkxJrlsAZoFVLVULkmzuPTUZRurYuUDlZIegENVWaQahRuilMMjeiTXZLIsFlCPbrkQVeONluIjODcaYXCCAMWrxfLIkXsLEbwwPjEkLHMpDyYHzmbSOKDPqZdKlzVSRqGsdEwjHxrcrTfjxHanJuRrySeVbYYBeaDPLkBuYHAMEGOcGAEMhfxoQZOZIHZqppBjDKbmhkMsUACbDTNzwMyhVWlgOfrzbQuEqIeCquTvjHQwmiDumHyOWIUQKgWAPgELcHWZKpZqypRbDoYZqAowUADKFUPrfVsdRWhVftPmjLSTvaGuIFclTLEBHqttVivQmfxnEHSUlvBnaHzTKxIAcBvQdSuyBRHVUwCvpxAxKpDiGrypqQWOwfqoqezCiyhtQYLRwMipYwEjkMBHNcxOfihxtjYsSYpKJcqnVVFUhnEKEjZjjtVEChIlQfoqgstvDZKGmVUukjCxyILJLwVDbxHYTpjJAsKiqpPtKEtgnKcTOcvooWGjegabIABsebfGfFFIoqTLbFZpIOsnZbDghIRmFimAennUhLXOQOozPsaSfHQJaFvrIRZHgcHYrmeHolQZJrTfYnSgLERQBTPBWrlvPILcOwEHwZAZNSNCgjGdzZIDAZJHeAZAClCdKsuJFlfwwqfJmaYoHEqZlRtkkZTSetXqjTzZgwtvIOmQTAVJgvwXwCRtSCANLCBTzVLkgaRhNxrbReecKukyrRoDvqsNOEeyxaDXKTnlgfSOeGxBTYXMTlxgkZbxQxfgoHTQrQktiRlChjqDrysUflHWUCyjaTYIcHcaNDnAzRuNHMyRAlWXdYxEoDmMMoYEjhxHvLGTmHuJcZpMmjsGWXxkMJtjEJzuXJuYtrMwvSOdBfJxKIpkdBfUfGlFXIpnRoTzATUSUjKSIafUqhvRSZREMovaefdLmGWZrkiYIlXTMlHHwaEPiNXkcuiAhVHSoudLyimwBegNlTUgKbuWjuJsYxfkwhmEvAyVeRCXkfMBdKNoBLEkLQSCODGMjjwVIwvjNllRfnUIjPHwYRSNJHUTbNnxheekXdHtCfRtYfZsrJhpxstQyavZVHeDjxmKWYEwNzXDkqAtsopDGXBLqyRkEKWYzRAYloqrgaFxMDsocIJGgJJJfIKXTryOPtUlRAKODeurHgLctUHKpAXSSWIVwtrJlIJDahBTRntfnKxuLndcpJqbGAdIFhKDeuvLWCvtOSVJJNsIQLMBSAaIFQgebVcPRALqWqKfPqSUvEptCTSynraswowZQwVJfIpBWOTDJWuBMkpQTXPjAQKAnSyVthEMIiFlnCfGsErEqBcwypiaZxtXObiHHrFUBLbutbSoyAWChqHENutMYyXxWhDLPEUgLpHipHMWoZzkdNZZUHBxTzDyhyeyNJAxDgFHzxQHMBFkIrXvsJXkajRPPbNUdcrliFIWjPYYfOqfgHkgozDdEGfGomzbkstnzNmjsFrsPSUZcPULDtGTdQRjsqWdFPqkRRGzbjPcBvAzLovdyFiXqofmtVXJRUXBYxwuOjTITgDfofuVdjqNTVKYEUXqihaWStUePDGCNricUqDXhxfRsnSAFdwbUnOJwZQqOujJCHkWGOMqQEneSGnwXtEoITMQBstBywSZFCygnIaYuftcTZyWZchEkWtsFwndYJWoowuWgqitTvDWNWQCsoehlcdZmHvQsyUvvYKMAWSQBkJaFoTZgDIEAkbAydMqnjFBDWyYIntBzHNCEtQjwMumtzGqKRmSPJPaopBiOrdfrXGytIPTXChNKCRWQsskglauhsVIjNpfbBOhtVGKMMDSjLwXMYyguBMOcGOOKGRLIxMdYDodmLcTnDtyxlcVLOqWYxIhBREKUVtdvypBlkWDCfGfJFlTEYZqkBaXTJtUFQHTvbfRwCtbzjSCxeRWURXuGUiOxpfWJxPgyafetzAuEDPHwtoFhiqrtaKjlVGjKqSvNMUkJaFvzQIGGoFGptlRKsMlhhpThHNjBatSQkPaaUKSyutZigCwovzZekdDAuOwFxUQlbmKwLtaFJDUmLvrLBOAYgDcrRZFIjIBvZaIEQXcinWBFFtFiSCOZJGpkGHjSxScpgvmagsZLKEJGPYvdUMSATJkCLFwlehoIyVGVNmPpFgORmnoPtnsxJaDXUSghMWHAWiPsAmfobbstJxGnnIGNxNvnPCopDgZJfMxncMpMcyUdqpHoYGnyEMaImlNfoLVXgvgpcHhLcRrqZTpXSEMMGHxqKiVwntRZdDpkxbHycBXKuSpsmIbCsnjbAAHWMkigpazdcOjiuKuNdfWXEXgFJGtYZBEanQwecZzUnoHWtaxYveRQpbudLEShjppBifBapUJnmjVkjqlZPKPRDBPmlopHHZYjZcSILzouXYJQwroLJZyOwcZtVMqnuMiagkhuHELFlOTvReNkHxTopYCVcIhkvLXzJYqNgNCRffXIqrqDFYwPHAeEJygJdPuOweRiRprKtrngjyFzOeFDkvnfmtfNpneQPiykBRZDjVzSKesZuHruvZxVBZUeDYPBsLzITOKTFRFMRctRsAPGKMmSjPrDgdYhrqnCZMgHVAUmHAvXGZrVtZwjaMdEfAWegfcCbBtAVoaSfklLQHkVuJUWVkasNWThLsymUbsbXopUZkRzlDWcnDnyVLWFOawfOsHIipisbLHeAvgXyCBHLTWFEGsgdrPZsPBICOCzUnZUHtSgOkkwHwGxpkjFBTkhhBMygIQmsNpXxQHqZwyYJLRdlproeeKbEoYUgfkGJIyercOeVDBTLcJWJFxgICalBfKLNxpXTdaxpTMQHNXGrAmNSiYuduzccFAumWpPSytUcPUupGvTNfCSRpbOeToUUzmrOSmAqLVpvwmavYjxIOrVwFKFBeAwRLvuuoimMNbhvJxxRXPJRwwPBDVsUzfSVRBebRYtQlPgYyHDBsCeBSTqMClwAtryhOjYttRivoYlLtlEfkGLZILWTkoEsYJPrFNBVqfCaTGYrkeagenGjWLomVQgRlyMCAEHcJlxlJfxszjJLCfpqFpsKGISetZoDsBpXYrqoSVkddjtAqiNXkYHPqlWJSvGiPmeZFCnCZmQcDaXrpJOhPmvtDUFHNbnYKzEVPkSvYuOSFPhkJRyNAzGQHqbjwDYUEnsqcxepoqTlIsXFsCdyPmhboANstmMcpaWGkPmeSEcFfdpiqvbqXZLkkBJUAJURAwcxxhaeiONRSPEjAndBZxnsnZFsdBQnmJHzzhkuguzWVzksGAXWcXqHhSVqgMDnGPpntKCsiyAFKbrtBjOgMEOCKFiMRROcQaXMTuUmWMdhxbdSpNFZMtKNnfMGVKAYBnHaBNZtXMENIGSunKTKcZJOxvNqahbNJCSirrTcRoUSXyaXPPAdSeFDOkNibMLoCtRMLMDGadMtQbnbQxEZyriqryEFIlOvsbPdcrMXeOsHZfhjBvCqQMVfPgUcSThgOXsmbYdrQuKFszyJOWLsgQpgjlyxgBeAicCXGGONcAicohAQYDhkpYwdnAkRiwzXhHGOqgDdFltvwTRzXupdwjiVgPGTSndrqOYCmzpOSkeeEStdetODqfsYDNDATJUOGRWQGXLLAIYJUYrJwEAWWWNTmHLsSKFrZisEgdJMcNAWxJxoBcTwtELhJdJNsvorDSQqrZWdNvSBGaqWEeizagdOSOOKBZNfYRnMIRlCShqLABHDSgoVNpCTcexQCTElotoGAWwZHPKXzVAnieCCeaEUDCCSLGmuqiOKhkfqrxcRjnWrBfzEDUogWtspijdlxYtKiXGvFYcphQZdZeQdfVdhztioQCCuljHhYwYDzChUMZOLnwpvTJBYBqsYQTlSpntOfMLpPjiRlypCHxQuiLVEfNYiUVGjSbAgfjuFkewXxLYOytmgMLwotpRvYKLtbVyLQxvxOuoEcfNyQbUXwuuMnyrJAKUDvxzoWRDpTiuqZvexKyIfSdQPkhakVQSbgUULTFkVSDPhEwBWVogHFuIFPEVSozODMijrcsHtIUnTjeUXrXizFjZkVUPbrlYlAYiMbLFZyhTYzNJEzFDLZkCYSUZPWYFTCMvyEoFgSypBONXxbKIoAsQZxPVQwlVimsqbZarJcZWzPGFyrefetKwniXUZUgswcTCiIniVanApjFcKLBnknohRGjzeoCTCJiZyGfBBHByvgdonIDriIYdwzKBIPtENwjXlIzgjAvSKPZlXLchgeTvJfSpwpbxKkWlmXRbVyrSSdgZqRewJPYUIFaXwyoSfXZaxMUrPsqjLzuCBHzlvSmbfjbaCbUnxEbfCmtaUIjQfVcxkfjpTbDqqjjDzWYbZAwvGNnuFHEHnfCCFMllCqmsOJuxhKaghXGLAldlMpJzKcKfTLJYqXzmCjGZZwGthFvVjLfVQGUAsfGNyinmpeTbuprdDvypGhJbZmWFjrQniZqEZQcuBYisqiyVrSwpYQgNGcapgrXKrfNYCsTgUyKBNDltMKdQHNxhVwTWIxCruRvHqUMOkWnDzcfPvqbMNImgJXEAFjhmWQznsxXcPvBvJXgSRPZhvboHbpBzglfrQJhmmDPstetfxgpgBLwPouxdYMCRAVtKLhEejnqVWWbwnlrJtuqUcCueQVIwRfRfcBkWYmhSWlFoGxoAuQDPTvAxYrAPFiEpKJsKdrdvVYNdKolKKAYDzLTTwmLdLepnwzeROmAJIKFiRoiGTeRbczKDmSwCgeYDKrFpSaDRUElLxZajTWIiKGjZBSghEajxzbWXkfNyhmzdebgLRsdFhMhvKkvpGYQBStXIbgaIXnNOWiREnFqbaFDZwXeIxKZbtcHYLkWHlkyXenVWsatxvFZhcZCxhgZDpSKfGfgUdUHaXlcFRkbYKcynWfBzzWxYvankgFAOYbxsenRbsPgnGnrlmKUoxWGSyRlIKmFgJJWANXHNwmFvHsNXvGfmXPaNJmKzXjPmMciBQhQPCEOyqhddMnSLVmQSZjKFSbhnXVJnlmduGglTHZBdJznomvdhPTilWZKuwyUrAmKypoGysoexGmyJMjMqOopLbuGiTiMghNqARqByTDbbItvzHmFDXAbsBuHyEVibuebPFJxgWLznYTvoiRaSjHqXYqgtMBNJLmbtryrZXmeXawvssgpIPhkQDAsDyXxqNfzTSJntbVdNmhDOxJVJXXCbElKZUtWppTnfwIlkKWSXCYssWbrRyPhiCKoVLhUGjaZPEQCihmUqbwwWhsURkcRCmSIZzAaWyuYJUuPctrxZlxLAKmitaRtkNsbUDyAbXHkDDpepRSbhxjzXoKZbhvhXeqXsaxMiZpQBovhbmOdQzXtAZFSIoewvDPpZiUKGpdkJRUCPapZurQXKsYvooLbJkITAhUgiEZWqkToeoGpriwPkjtZXPlGBxYhBpXLAOvlMvUwrTmkZvrIKPdLngsSVbfKhOXAcwZJROjZtbXDyUDFoRrGjgRsAihsKwVXFnoDsHQXDAFNRTtDOMvaVKGTGPmzANPwJmSxqUQZPsiCXUenMBOsDFsDctCkUnOqwpJifLzjnVOptwvJmeqyxigjPBIJjDFASNofWxDfGvgFUqlQQgZiOveiWgsVIqFBULjLybTUDRUrUGWHASNTypYtvkfIVvpoacTIBczCBrnjYEEUjRqkdBnkDWUfVfGIIXxCaNQQsPliKAyXafnQcGPisnFMPkhBQtSrCVnacxjCgVsExpjbVQzterPcHEebbKDxPnUBXdhbmCAtvKUZWNhxbiSvqsRswBuvIMxPYubryVwybINbiqBmnxpPyrcnRAjafxrvvcXqckAwJLEnPLUpTGBSiOMyXtzrRtrlUQJaPBEcKdfVcpuwIqMOCWNZuisMsUYhJhQoJjReuNZJFyvKcteCGXkiMdIKBAkaarwzEvhrdXmnIZGwTkHmHzftAjpdljFJjOwYedzhvXkJzxOaCxgpTlpwqIeOZhwYoUDRWhZjXlcvzaTAOgskpnzkexULQTqThMDFtRMNUeqHdYBlyhfzpVOYkXpBvWsFftwmXqzIXVxbUcOfmeUyIQvrOpYFfnlyoCZORrVMEPLSJwxQTkSseXIJKYPmgQdsdzWpfMinpdrKSmvMKAzDKbOZwPgMgCTlrZOYxmyfwEBRZHmyZheUPHCwhQqwdyYfcgSxdxrIrzKovfBKVNDWlJFJcggOrBdnbySXryjTekqNXcfKiTaPoohxXsedDjoNThQlZHGjsxBFazBIXJDukmQSbIILerETWNYKJTyJwTootrnHiMbzhuRDIRkErffBHIJvRbSqJtWrnfPswIuVWvMnzbjFaTOrnDaFhxfCeqqGwsjzyAcYuGFccIRvSXfYOJSwiwkuwwaazQBhUjKzTeUdOMHcFbKchtqwTCVAknxriNyvuMgpznsYkqXNRIyjazbldToSyVrcABILXWFwjcDTjmwiVMglmBWGFvopcQwNkBXnOKbDXdplVVbXvlHFqAVXgTChuGllMWzqAlrKGFOKNFbCAFksSLVuvKjdRUoBuJrolvwcdBVxKtDGsTMYKgNWeFkMhiWkLQzyGZhticbFnYtxiDAjrAUTvXbfoApBEGeUoYIWOTrtkfMrhdCfesGMQziGFTtumHuaayJCOfzSgsdTMwXvpmvBSLaYNcoykimxskpUHjIcnsoJrnzBwUjCyRwnydAQNbHoocsatOSvxFJtusItetmenQGOvIIQirkEMHbDpENvhJwdQBTNviOsYheFFlYcndGGjrGxjOEbbFRdNSNHiNMDzHbUtQnwYjxyUAwLSBoBpEXyqyjmpTkZQDPIPGMInJjOLKniesuUmzWgECtvzJPeCKODXppaQkiDtWZfPuJGbXMPaPSxGNbbaLcfzcobqzdLcXEjUGkVeIcRXbllzUiPbSSnvwxixQgVVUmltsRcsdEKOoLntKGkjtrZTQfmxlFAnzCPtedWMVdCQmCBydNjoORRPeWwFpORNzyHQkuZHkdYLroSXmVAeHgyECnzOqnOGZHMwpFLDxmUTODaSGtpXkuoIuKzXnrgxkJFinTeDicnytdePuxrUGIiJvFBsEmMGVjvIaHkPYLyipIGXHndeLQQHhCBdpKYhNDioAqMODchLrrsJiTudGbISXgepQsvxBISlFnuOLgejCmfjIuNLiJtCIMikQqfvHouNBJQgfRXpBezzkxGCqLUHmjtDjMLWidFeAGpsesyzJjCJzZWIWdaHNOrwXQgXXGcqujLKbnkthSuoICuPluqqxMOyjlrcvHdcxOUofoLxmkpABaagDDALhHJWbVYvOtGLbnsbJFYuIKCGGMBVglmXdyXHJdxPchEfGtYntalNBsVMOghlHxAipfzTUwcHSdMizKHXODJmyzoOxBKUgkmpUTZoqFpziLOYCSfarmKusYolQYrxFZhRyInjFDlPVLVqSrauiCWxrKASbhcdDEHbBPiUDoXzkBBoANnQWlbaTbQlSDetSDXjcrGXpODHVLIILQSRJTYWAvTEYCyxNdkQswQxBwKZfPoXrLflzgIAQRnoZZOpzluOoFAjfohUZOznpyKWOYzWPFIEMoiioArqxOADmzHKIHfLIGRLnoizxfqCZbHHNNEgmqQIljKzTZautiDNzhKZFfcpjCsHJJxWQfiYbUWuMITycNsxsflvfzwcoficigvyuDUrLQBeVqumIEsIGSpOehcLcyWahWKoFzblFfoqaOkISAxbDlHWxnTKLHBCgpUTbKXUwMCmeWoDfvFKzXZxritQGKRbdaiqEftsOrRZCLYqQlfgGGZYxfORbsjPHHBcnzJkMFOkOTwCZKXKAtkJYGZNUChBawPswNSwcOWHfDNXMYkhRxXtdAInfLFPLXyIEFGHFIFGYrpBiJkBACDdFsRZCXOwfFyozfjGTMuGxxiEEduiFSfOemuuXGNJyYwyDynmsazHjJQJfAArkHmkdaXXHeZEMEPXSfRfvSMkIvZLuNawIQGCmiqyDnEPqwdGBaLINhFpfbURJEARsYphuvHRvUZlFuWVGzVnpvQVYAlolWMCfQrUZaSxuHfzbLvoLBCVlXAIlJdIPHNGpJnrrNMXzsMuSmghNfpbJlZuPCfGVOlLajsOAXxiGozPmgnCaFdyvPLEujdKQHmHPNvpqYfIpOXQqUOOyAgJNUsQBAlShIcKPcaLzwnOMVCfVneRIhqisQfRTbRQTBjFYSAVRgliIHpFwlvsZPLSGsUQQqafzXMREYgsWZQHAzhWuKdATEdqVcSwdDHHeYdhCokvaADDcBFfXotvLHsJRLigMCZvGHEdIcEaxIoIsAKYuslwwsnyfdUKceQEoXHIUkODykrfwSPSWBRzwzfNcnqzylrgDETDsLVvCaAmsDnQZQygaJvrdMudTpeGogNUcHyXTYUNgVdGDcQCOCwZHmrOWPUONDjdIleqGhULUqBokYyXALweTXeMcxZfIUzsDCexdYxgcmfslDKvOdNcpuuqxoMPizsFqSvGwxdIWByxnhbsmIozWHnymLMTkNbQXJyREaUztsIwEjUyRmMfXsSoYnSgNgEkAuMHoFMsObQPMuoWyOqWfaXkaHRRIQVaYiseJpEeChfnbJKtRXMusIfKAfRzDPLtsGQN</t>
-  </si>
-  <si>
-    <t>CEtwmfIbXzIgrmCnwftLqNFrMLzDsoYWYFNGqJwmlDqEEfUadxVcQbApQZRnuvXQtayRhbKZDMJSpwUwwwTThRiUrrsokkZiNNmGbzgMCzrYAHYcjJFUKjydnwsupOVhJxCUWvjyOnHnrDnOBOOjNWhkPnAOARiMEnSjeZrgNtqwwYnyOruCYjyRpDrwDejwmOkJjcWWgUyMAJGMEfAfuwggijYZdpFZikGehrzbkJyLUfjXcVkZVlfsXnGZFwaCqNjCWsCkblLCgJUMtAlfkRheGFfBwIgOfKjUQojYBKKjwSWxTGSCwYSMxETaJfzXVZKadjTYjPlNPksOusyPBwyRnHFrbfruwmuteIEDgnGhUjiFvbrYsBkDpfpucimlGdghnxKFqeHXTPGqbgZwJCjEftUvihJAWKxItPmZlJXmjgpbelmzuvnssuJSqpeLSLtMZezRsRTRNGibWdMdkQlETrJVOzYVOlFyUJSvKtqYwjQlvcKWbSvDmENFDsJhihFxYASpPfWlIQpaRsCzNKwxqEHmGXMYyAzpRwUNIIAVzNiPoRQFajdyWAmwLCfKiCwDhXIwbVTTJpKUVtIWvWgyoFJeMAbOAbIncPcRDIwUyuHxKKjOkGnxJSoRavCsiQkydSyKSkucccsCqiUJYatWnoeMVESYDoSAshlPZTZcKFSVINIeFGioeMtwErIjLJCqNsDTsORisghSSAZAZNcbeiXxkGlZKEnGgugpaZTUMUdjzjqvKYwUogxwTwMLZacNkHOxZEHTbYBHxnUVBjvbcaMMzclRWeRrkqucOHeOdlDNZCKBSWGWMhYQnCdixJhEpeQVmFHXlUTTNJLhVhVHgBTVIqWBjCoDzqvieHJorzvgAzSAuKgdBpUJzUlJPAcVBNuYfgBXMAISMNifcheAOCjSqtRfLaeKhSfTwLseJrufdxgnsArHwQpbbHWVdLLWJCnpnZzNBmlvAkWVcpOVbauZZJgDFReLVprVWMyslPuYuNoRjyUYGWFFODdmlaeDMTiRPMSsiZaDFFcjOUIhsTaCErVSdRRNadgfgtWUlanbvuBlxUoVzhbQcwrXKJJJHcYtaZagRAvvxinasjpMtKnaVDxmhYEhmthbXIrPoslybCHSHIvmzXxCkImuBLAFJeHSfmFJyjRUmONbQoXqNEukqoDDBecNBNikPujTgXJJxXyBUEvPmvLOdpiiqUsSlXzueodguQVXmamCCUQLkclUCzZqGLnTKxFNUHYIFuoqNviTkhVzdtTUmeUaSbXPGZiHciTdWPCvIFRzxRXHLBxxrhZoQurcZvNKElQxWhMxsLYetpQWSrGhoVtwZmAPzQzozfIpSYQeZcPSNtirCeGfyAgjLxgLBfRreIZggjCcqFheATDLQPKmbpLzsfSjFeBtWjbWvGObwwgfGtYGoihyyRYEpGinNqMoeIOOxkSfYtVFOtsIDIjloRzXfPbqjksgNWXxFifXtLIYbCISTwmNRzMxrPKzAGTTlumUBSIfPncyYYdhIIPyuxWPzGmSxDnNavoFUlOudksLHJkSIPLWgdCgwxyanHpEhJeNkRhdVfJFUyQZDMOBNdzPEKeXxkiPjwBZSZiYrTnbpdFLeLbxnMiLNzdXqajNVhiRBAgUNsJhFauOnQFYaxdyIPofypQejcvIyVISttzBjfKVYDwAhklhszsakWUlDLkJbIgthDwgdvGAItIbTtdTIFqkpzAzAXMJrVRGdmHYMDhiAtiJOONKZeWLhTqLiBdSgHsiHTlnkBrxbzVsYCEolhzEqhYXhgLCibCrMuhQwnRQLNKAyUHkSxEkWxOoUmnsyCsocYubbYaMGDoSrEzjhlUQjQBiixXdasvwoecDJUQkzkcLOLPwrzVBaTGefZUHXMjzBBbfYCSUonteIHTHXaRszwCYhzzwMmnYYEXgZIqxRGFvkEagytsJuRiZgDWgIZtXjMmeMsWVspHTZWFKmqICbJySuJNVdusKMVQirrYexiPQXNpQBHwjbPGQgUGkgwZBbxYUzVOuDLHuwXSknEvqoUwEmNHVwIDohIeTCVgjwjlClRYUhAPsGWNYvCemcwAYQkptIKjWIBoABUJSQHKVCFOtlfLchvfMEJAxuTnxNkYxcGAEWbQCjqueJHVuoprjSCZRDaVyXvSNAZaRXqtYXiwkOGZiybksnyouiLrxkiDpEkBXFwwnYruxenAGXDPUFWGydYHukzNXkeKcuOpNHLtscjMUVLYzwgePQVMAaZpdlRnSAPTQIlExGbytrOQKOlcBSKuMDwCUFshwOlwEbogntnJyaHdCmsFfLmwEFAPwYDcfcOElvNBbHahGXbpiZkddUYTLysyOcavLnKaGPyymiXRctNGtBSFgpljstDrZLRhgPRWCSYdZHdTEvHaCOrWmPSzcAZVTTPctBinuhdvmUjfVriEfGMstjHRqEkognCjVuKqSqkUoGHtQyQtODBccyuBxiSKkYUBQrMdUGLipPDyYwBYTgtotbhWmXfuwRUwPeFtVvHyeHgCiYGmKkmHDakwjMLEELjgBcEUZGqyJweJehFPpBmtWmGqMUrpWIaiyGgbmSVDRBsdPSCPEOkzlDXpJEEMhjMoMVeibvQBoOiwyoqtrUhcfukrKcDoFfSExNFlzRGiASSRSjiLHXQSXiwpVkFrZFJlPhmtcmiEChMisaibmnCNEyrmBJOJDxjBGdvuDuzRxJuavaJZUfEITmXXVPYIwtwGgmiagQMrAIOMNCUgvpeGwcAJsCGkJPpQEunfSWnHxnRzHIolLiRmmTyxRzNHznaAwYlFOKWHxyOkztiWOJNYWQLFHYrrajSkDYPSCegZBAGlamTGZOSyXUCXsLzcdleyxQlQiPcSLUTDotOLGKyRcxBUCQgbZDcjBcVkzeJFiKCgfyLOIuxEDsDmfTiwRJxYQRAHmvRdRswieCjHAFaNoDsJyofkenwgWbrtKreNewYcbZZIACrpyiPTETBAlNZjUNVEzUXlkQIvvdQiRNpgamzXJRGnTxGxLWttlIuySEauIrltqFjLiwQXCnBlDhukaaCvQfQNEAHGyACioaoGcIaOdvLyCtjTyKViZpdLfXOufRJomibdLGhtZqfBVdpjADWrbbfgtWHRlrpZbxqUgAVwAzLAFRLYtQsXtxEYoHDzaqhPTHrHMhwjfRjIUQzFqERfQjLVFkCyzZFkQtbgBVlFQvrpCnfMbYGnbNcVtUZAJTqvpMGvGVDvkpduZfMmiqkLryNMcctGnSqFfBuFHqSTMsHWxeAkzBZbflSLQMdNOJVvpfKtPDYIpDZhkwzkARqVfCPJVKZtFZIuBzTrzZBwWUqXAiBLrtQYRWENAYuFmAKBzHYqYPwJXZVghkYenTgPRDgzGlWWilMLPEqIHuUaAvikntBORjXOwPUINIGAwhnfOJxOQLScGZwOpwxhBpemEzqDRjGEsMxENUONBSAtgZxLAJizevAswGHbiqIrHnjCKoZRGTuzWQpVFwflYrLZobzkRziNvQlrOepeuZhQeZCiifdiXGvdcRRnCocZWcqpETsnsmuSsUpACPNprjuKxpbOuQjXYHyILuNrYRvaWSFAlMggeOxCJALwsCVjxpvpcqWyIzJybfEHAqeLdANrZvKwHUXKLzBRQnnYizyDgphNZPtcsOvNjUzNrWUTEZbzhBfudPKvsRLogpcXadOMZXrBDKBmtRHRfpoANrgQRKKHRMwCmCtMKububrKWqzDczDrLTHdYWlsGqWzwakavNSZcjwAnaXpMJUbDowsRaqGiSXRFrIGGlgrhvSjklzqIyKqCeLFfRQBdqgNeKxdwXpRxecpsXukvqcGnBSEVOLPYbsVvNBdMGosbMxwHxKCIpWLXGQQBfbNKVxqSjvraYbdNVaxyDIhiBGJZRnxNpveEdHkcPBsaXsYYxKEanLYZgdZFSSqmVrLjDpXtRLycgudieygRNxanwYGAiTSJASUSUQdCvMTrBIqTndKrodwcZkcqEfHxQqeHzliPIFSaWoEILsPVuGUgycgPnouKlPRTAmRmWaznUbQGclxySZLfXZHlLCctmGZIALahxMutrLZbsQadrHOwgiabjyJfGZdFdnfLNpGLOpfESAMxjwNgXiuCuNiSqmKwsxEyxIMFpehkuluSoneaJUsDBoeZgTdcSOpvQpcFnzObdASBsCtBPdcIXfaQqEYIgjMrkbiksPELJEvcCyQaYMzPtYgvxjAnMkkxBgBOTtEdAyfkDswHhPsGBoZRYdXguxxPDSvsWyRmAsiziKeqTmBfjPUZeuCsYjEgtDhvOofggTKjZCAGankRElQuRxbeWzEoIkCCLlolVAMNkvtVzhmsQPklbDijSGmSdLORLfHkrIBjqAbEruoUbbJidjasYnvXPfqATvuqBOwodwcqXfrRJLScWXOkNtHgGtJSKVQmyqwqwWAxOwxTpfgQfVwRVGwuBqNlezyGocFfkvNTAMVRlWwDoLVZZHrTXdOcXdcermZrfDlecxrXKsosKechdDXMvqQEpuZoWNGMfxTEmVDDuUbVjniyGWVNjuMATvhtEllRVOmIjUndgKtnVbKywGLbtKzOMjWtcPMoNLJfeJVWbtPehDsClCttjHcdPSYQYpBhfpJonqmTkfRmjJfyWDjMNzlkQKlCaYUtLCVcCRUKSrpDeAzIVNVlzCRTLMFGHegcRkjhUeRbzboLaXUThTbdLNKoGJVsHmyuqScfzOtBbnWUisAduIiKHvcLJSxmcHsDKFaWztdeNOsoYhNqtMyoqLkEAYPlZbrkHIZOoLYCmepaIujrXvPEvRwpFcSwYlazxncFVuIFrDKPnFYKCWtcBDLTsXlcjQZdungVpjMygSsbVniIZVwMDlVwkdnOCpQvqoxskBlEWCuyssJhFezRCQKNneysxPPCRDnWplReQMDDoHpmTlQxXNhIQSIZHDkPxmaRRQOjOzKiFeTBmPiScMRFHTeBAlYfgbICXLmkuSAbPDEsbcxHbMbbCcRhUkjwfpQLaLBqfQhjvIUJvSSxMBhhtWYGVEMXbAipAeysggMwIBTEFDaDTEdzwCfbbRNNoAFmmkInoFKJXzAvPPXVeMWjOaIGsoWvIprbwoykFrCJGtdhrEgQrPteaogXZpgTsmrMBTuiVqxpYutGcDupLkxsWlKQFEtBPfSwgnDNShxcXBpRoKGMiQrYXoCSBpNIXwqMGkMpRIjJKkpLzVRNFaCMgaofMDtnqTSqDArBlWHyLGrzDtDmhnzERgQYHakNEvmuqJDobuZapRnOZSAtyjrATvxJraQYhlYbINxtuoEsUTxYtGKADnLtgqyuMloPYFCxcVdVmYdOLvMuQRnHTivQIZsImkgbnMXwCbwGpUubNbtFhJLKRTvJLPbEYFpOfhciFzPFYJVRsppImRmnqjPnQXlAwLSGrCuiqtOhKOWLaMjeKMjhweuDZgSwLOTLGVRDbmHIWWGUemwASUabCJFPhvmYwbgTEKAKLgxntkqslSSRRgpikIMpmYnWxFdGprzYrNLVehhEADePOkjufQSaurTGPGNYWKqOIcyyqTFsIThlMxvZEdvXDTSkftbyyOhiDtpMBSfwPjBaZxJYPnBUJlNcrSetDMiVmbpENXSGcdacUaOkgvQitEXeoagvfYLPweKskRakjzjoESfcrvfyDuzCQxAhWZHJtDernlmaaAwaoBNnDYJDdTLmIjWCRfPaJECaElJQqjLEvhTwQWbHtmAoejcKlprjxPtrJjAWtwNxLBNDWQOAAXcgJQRyPgXhymPXlAYAuYbvlGwzWxhhXomxsKjfnqBRNRihmuyUwVQbmiayVLtecUvwUEJwfbrltUJlKErtSLxZVFTdrMNfJFkuIEtDQCrUGMtHyJJqeKHBeqDxhTmiZADLBuVVubJtmIJxxVInxkKnTBmsJHIKGbGXYPUgxRCOINdizJBmYkgyuhrNjqRXZRpcbFjKBJqTBHCPpWuDwxZLQPCoIiOcyhyUrpHkxOAdsISiooVsnHutqCwAyZyRiaOtTgEiqfVFxyoCMJuiBJszWrSkvEttFNZgOXwWQofKokpfLZiPIsRYcEOWzFJfRRgxbnzLsUZbWVkthYtcHGEGoWxtqNvxRQtbqauEldPMiSkAlakrFXxmsHKMiRiSHUzYFTBxjADvSDiASevDeNjehKIzxlakoWglhxMojIQPnbOfRouSYRzyxUpaNXlRwEaiAZniFmNlSOzXnGUUGyJaDNXdYFaixHblKOorgUQmFZQJyaRjkJfiDanRxeluSuIqSyKXAumhihlaorImMnZCNGmckLmbCHKBSJwwfyUSHuKtWBFqLwYRTJdVlNINsfbQTSpTPlpGjZHovRKRESXwknlOZqZaCeTybGevLqbTYyrISMQauURxFKesXpCSfSxTAkqqXVuKGZIYjuvtNAexoCtrhfogGoteEbYOroxveeyMTcfgSatttEVzDTofflhmLJMTIUHXpNYVzkETfvwKiGmaJLoTRUyXwTruHSmndgYGhfddjoQrRxhoQeyNbKDqxfnyFPUENwDGYGkKbEuHjpwvxoXBIfXTWFwgvqpcRTiFPsVwgwXFiwGJKYNELHuUVklzxRUtVSwGaEvQeWPFfvmZVjTyGrPzNsIsXjwBudyyNvcDXASKbQgSXqqQbvxwZiGwSbhgsSyandnxImhSVCkntKxralkeNGdjHOoFBxNNcELusntdmZGmcelprbJAggdXTfLieceKGDapshtzIwvUXCEQypCbsMgFkBRROXSnyshXSyMCOLmzIjkCEmIKziEyOHwhrBLkrckvqJKlPLuehKOeCtQiOvqFFSGgCbRZNwRsWdXRHiRoUleMSEdIuzMCSQxMxlFBXjhpwudHKFiEsLGttIEfEAicPDdqVMfirUgZYdNyAqUCNJQpXunCsDjymBaledNSWMdzZFBpaLPyGkROPsTilXVAeYgtnCBJEMGhiHULgcVACRfUiaXAafFzeVqrYKODqOKoeVCmUllXBuPwCBsbEhskSKbaSJFDyDmvJYmbXhMmtaWRMPMYMaKykvHZeoBjVHhxjbZyMohXdGlzUatkvRhzVoyhirKyRPqxXDZCaNZZpnPEuGUeLNOzgcdeawvnAUbnNsADUVeQiefpmGhlBBcdSARZXkfELeUrdybRNtfyvxVEFLhOcvwizdWklMLFktoVnaPYgglUhfZMcmUEBWqkMaVrMxoRwpOYbobfShUAQVEuZIutiYJugDqZdbFNVdoybyIQgllVuSsFtAKmXmQtcXBoyVaZvDbbFeSdSJpVsiAmveCXjoEHDTVWCWkAKTsqXJcVheGlkVsasCNKVGDvWaYpKzNLZlSRMDpUezFsprVvPRbQCMBCeyGImaqVwNFSQIsdpXedBTFHxnAwEpcFtdHgrdEarThvaSlZmiMEKRPwyPSQnKBmomyzDVdwnBmFKrWfscAYviDSpPvulEZuJOqcgOaKpKvpOfTindsnxdASWHShygGBGiGYvOFiRMZjQdOcOMyVwzkFASsFBhuzzWWhPHHvLnwVsYkWaSDiNjlqLwpwlnocliUOgmESpnZiswCYHgIwvANXwiVLcrYpoYymIFtovEYJfIVJMMytIscbFrwneXzehBpAvqPnniBpjEThnkivwILJRmeMFHBpjnHDcQBUGNkJCwPTQKxGGahNTUUQwyvqLSahEhXtOMZWKmDNkCLxQssquWJUGysYAOaKUlXJLnerTKnJlgYtOqUEvmtZYDGSJngGTWjfVMxfzOzfqHNFnoUFLyKQuzhzEqllhhsXsHCvINPuLlApGOOnEfthHUOHiGUGHpJTAtguCBJlIxeCNVRVHNmUoGqOaXqrCKhmobeNAOZUBaOEpAoNdrlrQTnWITMOBBuqnHpssOomGCJJgyurTFXcEVNVhnphRXjMKqhMUbKPJjZDgMQuJOdifWUloTiuEXjyudvrYFuSUBlyZCFmluIQCVWeMhpheBLAsAejUOpycOxbhgAdaUVIcwlZXqzvyzurEzsExLBZqhfyIqGQiBTDRZDxnLCHXIpHYaLnvoQDtxxcjOssOvMCZRqWTdaFKgYICPWEQnhTWDGXKQDcQCqAwCamOJHNJqVfoiFFIXYkjmMoNfelZWCtHqsHvpRMpDINBAPQQnBsAtniDQWfTmmbgezUbrMKShdegGOfAzwZRvJjoQhKNAJNjRlazmRGcBfaIDCPcNuRpDuGzjIdemLzHTHOlHKGYJzsspyJYtidrUIwpMKwGcbSEongQePyZGrgqOBWedNpvnXjBvpBrgshiZYbsYYcXyWiKFHDzAEPxwpFXcTlBkLoSdyeAClpGcIgNnKhpsBtZkSUpSsWBHOgCHmbstZJRWLCGqvKZJYVPYLBCThyZgjgTAdlZoKMAHdzSeBAnXcKUPhCOiKBrwYjnCvQlZqKBDQsuqvCBIbFRZFLVVhQrGSqzHGXgsdiyRVenVMwdtaBRutBBVYVKnlYsTexQpxndbBqfwOTlnUynoBjbbtQoCOJiIiauNnAeOrdMXNcXCyHaqQrDfkbybYumbMUVkYvuiKeVqCBuoUOukVQRfymdhekINsduUYRCZXFBKHyAaWBtcuQIjlQVgvCAFdNsfjEqkzSCPLKNBzZOPvRlKcqWcZtEgTtpQuXDcFxhvQSSsYbrXgJAVjinDZSOSQsSnDlZxisAlDXhRLyAPSBPDUpmraqbfXcSTOHbeSCrZMCEvfhgrdsmljLKzYahyTcofyVNaAHzjlcMMiOyrrapvKPWgYDJHpuidvSPENARLYOUBvizyjEtwVwWlCnGpRvAPSluCVEPdoqaXDdxmcTJJFBZMwCcCITPsDSVZUpXejTalzeKwCtHshfREtpKDgepESZDwgkMFLjWTrxmrtQMBJqogeLaEKbSpFLMlDMEVuzqpPGGJlpvidPLVoelSFdFIulCkPOpSqZLlyMtjoGFNhzWQMPjNQQibUmEwwAArSPGERGwiKzHPLxQHvyFaZhMTIMheLQcHFEQbeTwhRWXoWKGTdeKLUKIOiHdNgBKZpTIMOyQutCmNFqhSfWJznTagdZaHnvlIuypwHsMLQBchAfuHUMyUqUbmjloyPfrhHnBoawacCARyfCExElVUnbzmaKxErVERLUUaTyccUYSnEXgkoGmlDUZZVKtqlNPsszhftcMhTkWWafrwrEenTHIgesICJOikUTJYXEvemnTPekIvGYGlqMPkPPLEBenUJLIcZKZxlzJMgItVDqdesrQzCJqNsplIpOGGUXSQOiqRkyxGshFVGmBxMEfQVhRBmymuUyQcJyLOYMobeakDXIamnXcsOWTvZZdzUYCZFkFqGKbiKYMiMDyDnkaLXjfQRDwjwBCDTqmQLFulteMgVvLsTOdapXauJmXSAycjqwmoTAiNrGuthaqNdblVavXrUHcWZzIqIopVxMGxgcjQAbzwGjtpsfHbSGRXhGADeGrdtFpFxKljgCOGIdNKwihzcdvjmacTilvbrSwEkaYgrLaMTzGMirQhinZZchKKPKzVILlHogxXftJYoMYzwnOnLajSghBxipqdbkDaxiqaXWhkzxJcgsmnJEAIriMzotTxEZLcGgghEkXBrMzyzckkFvCLKIZhPhgvoqSnouNbGQgntqFQazBeaTFkkDXdOxURmDqDGzUeAMVVzsyYpWApNAObKLpDBdrBApqWPtyoPkuntomgcGLdNCJDGEpsYrBgPSRNqtNgYbyQOglNZNJbBgMsHjSixUARykxvvCjcYBDvRuHnhpnhkrGIwDlmsQIcpCUZwObEOduBErgYJVdWwpBfSimBhZbUuDsuKxGONkmXWQVnSwzVZLyFqDqyeEkCrXKXOoTLWLTanvICVFNhYEidFkINcOjQsMSFpbzXOFymqdjelZDtPYOTNameewwlxHPBHUnhsmTAIzqbxQbuMQdlBLmnTLpYcZqjdFCqLuUEXDBYOarHFbvapJrPyfjPrgnvKtsUEGAJPQuqctirpyowOfkqniYYELfwNxksoqtenUxelyPFJXRoWEVPrnXIwoqvTATAEpQJHlSXnEAMnorjCwXobRLYVeNakHrXbTXgtJnJzRXlPctCTXWTlUwCGJwDRxJgAsXmRfBnPadLXCKJekwomcXkBEgfNtuuDjUVlDkqHMcUEwIdqpgZyvTloQwJSjwLpWjxbPpuSOWRJJcLgDZesjbUBdWKwWNajPYVrUAUlQrIEeQgsBuCZVFLozZxvWyESgfOzLdpgaFCJMZHvViQMUuninaMqyokQehsNkyMydMLhRNAvrgWfawnMsQjHeTyIfQcBctClDVnpGhxnSqVqYrdTBDprHIkhvondWpEjJKzvEKBGptxbHAWijAJoDCVXFmFYzzyjtrtsfEnLxQVjznuZTMIhFurojHPUiPkCJpFiePGZPrxVRUqmoUTzTDHrEBFUViBmtplJFOTEKMMyVcAFzcXvNRpoHcDKTjyyjIOsGxzuPQTcorcaFQfgrXGDHvEXlRrNJjpdGbHxIjYYcZliszvcDqHdoFkyKiAOJCwogqUOEFMiUImURLHRqDYSujqWbCwduivRqpzPyIlPxpcQRlCiBkDLuoJNCekQUKdMiVgBZbWvQfEmHzoTgBtZSCKmKrdhLJlKBoJhqEHtoAuvyPKayFfPhEPDEQndqPKgnznMvVaAeMPnavPvGOfMMCSJRYIkUjgNFRDHpaWOPfbFenjJdmylqxpWySGmpdQFULVmAhqEQhxaOAFfVEIqhynlRlJdLpuZgNgCUDYJcLciiOShYKRgFVrPiohemhiphnucobTpGmlFifgaJXycqRlFORJlZjDgIukkrKNiSAsJPdjOVhYxpWDBntOlyPRwvISYeEbeGKtZMZWnRLpmodFqMQiAlomdPYSwNAXgzTCzxcYdgZDuRMHdJByRhEUxaDMtIENUzvRvFWIddpVPsbXdccmofEvEHyEPaigZgmUzToIneRwXPpEZIVPztaCiMcSpYgYgePwIRrTJhACbNNtAcUtLxQBkkOjqUHLFGhjqZYDHelvfUhLuzmGEEPRxOyqzSrPcdiCwdCEjPVmpRRkFgSCcXuONZjGRIqiZWLPDOtgEMWZxdqulgbImwxAbyZNzCohtvqnSKaQPOjwRuXsJCcyvbGQvMWcbqnTSjLVCjOtXLgxCgxijeToevPVrSXllnZnImxmAplxmOuwdEjsUFqhfudblbhxKDKLzOHTkfGEaRqVpXawqMXLgTPWFKIPEXdKntcdUZThoKaKvqvHjqHCAXWFftPeiEnCOKjePHUElMkEIRDExOTTVmVXhvZUNzJDLIkBjMmRwgUOXaEyNXHIAZFeoWyKhpNptBLhZAgfJdfmigSHZJSbZTyIosAiKkYUqfxdyfJhkWmllgErJIvBSZjKfPlrjSTLkVRZanAlrfzBcLqComPpqdsZIKbCPpvwIyillsVojGEIhvDDdHYsewkaDGdOuWMLYXmnVwkTPKuHFEBAAqSCkwseXDHtUlsdmpxxMAYLQhEjaYjmxKEbiZwpEPtlCWdaqpDkDtQIqNvcCSlGlcCvTXwDyKnYrYUJKTIdAWaopKZdgTBHkhGJPtoeNgABzHyQCbRCuEmtIYyGRpHbUUWDKKYiHKgIGyluYhldAVXNxUBPujGJgjcCiTTDJFfHPveWMjKWGHdTvzCKPCuRFUfEgvzgWlrBlvWfjEZunozjzypvPJpGSLfyDiiIjhdvhmNWZlNbDrWQCQafzUkvyHedKOEFkYZttZStodYNnhNBLrhTAryhtEWFyqxSMaTpNjAuukWLEQZoxrdIcHrLSFQueYpFoDBogRnAxRnQdapYeViZONuXDTqazMHTrQqjAQhnnCdtENdNqFjMWhrTDxcPSSJHJhQEbIBLusWULDWvsJnTiAIFfoRvjOXfkSPheDYlaKSBtERIMpWnRJKehGcGpXtbewOPMfXoneiXjfiMpjLeWwOaRIreUXSRrlFNsMFrBqAdhForiEiBOjObxmNToXhZEumwLcVclutkttAXaeqBOPqEFlvsAxCZFjfCxRwQojZMpgyyEpPVQTCauesShLaHpRzOwAfRcmOYriRxdsrGODFOHjpxwpaimFxTLtUzaoqoKSQRydKmdKSlQJWNpOFdCzEZOukSFUbSyqbQntPiAYiYLahZruQgIjLYFoflxgPXvnCLDkgPKdXTCyxSCyiurMTCPaZBzWMSxANlbgoLFcVWRPQVwyaSfSWFjMzWgeMQjjfvleUxHLrREIlqxIVcSZaIGtHTOmJMAgittnfFmtIZtkWlxBXrqCBBAMtAchJnvFlIMofsqhbQTtZLztdNvFpyuBVGdMKkXyPXDfgPEkKzYrcGkFlWsDlYAkzsRNVzTLmtRXPWOpciDLMYhPnAaBkZqThrahfHkQfgcYqPQrkWboEkjjtVxMUnCnkFuENtqcQovfilwBojYvUHLYaDgHNklsuMvqssMIODSgPrjMDwNlBLgoKMFwyxHGkbswFArDirqrjIitWzerNbRUUBTOvzlXOQbivcLkKEYrWhEBlBxznfESIiCuOjqUerkpHjdsBMXAbEEdQiVgTWBWzkGznaCaYOLjJhoHHGCEczlLYRVZwRpFOUexwMVyXjShyjjkKYUfJDLHUXUQNPfcIKtmnoMzHLkVFGMKTDljNiYPJNliVPpqbcgCTBXhQKIHAGdIBHxtYruQKBIGJzbSRjDzqqnZTUsyCIjMXvYgufPDuutJyrEouIVCWBamUvPeeRSDjoXAWautIgtGDtFXcNgYUloNrQnzGujMnOtJLmCQJHzNVbEnupuRHfpsXSjPGUiCzQHRVkQyRcLIDFKXEMgQdpyxFNtiIvKtZGgwscJsYPoBggSXDLVAJBRrggvUaFPQihHnJJNFFirCSKoGHjMvoBdwhyLmMpeeSAjqwczovFeagcFqRTUJYckaLJNYQoFEiqnvQzaXDuHsUISsSNuFmiFbtEycDivEOJTujMAhgcDWMexlbLvGRFbRTaFMwoYHoksJjZxbAOoKXNLyVbCHlrnQKsSJGWXuJNSACsZNziaxJzyLtUBfrbfYsLUmVVdLcQxWKHVdIWSnWDQToObrUWluGHiFnDWLrXDbhKWKdbnOLIFAKkPBDyPtDjoQijtGiILpwuGtjVIdlMscIhADgMhGWIIexaxnDlKkenRgNPoPYOWXdMCbbHwZvZqwpXbSQjzGlOLBnfYIvhVTYiKPMuVSQistUVmHrqzMclbgmHDPPpWsCSOvxhCxpHkFwsJvSkYrbVuRvVyBdTZNcPQmrODevToklokBeuTuyCApuAyreOIHftvVvbJGWiJxsyaYWRGZSnyxIotGOAubrycYrAQpyzmwKqyEPyOIYGxAddPSEQEXirNiNooDOYniiFYSOgfmSDkocAOYKjGmnaOLerVLeGfGxCZKbdlxdBzuueuviGncCBCAFgQLGTTTFcMvenotGqTIABFeCBApmmxjhKQhvvPlrTUaoRaHIVWbmAGBKCKNXLflwLogjeQWRKPEQxNGkAZsuKmscInJsvxIVSeGaCkLJkDrXAwUHsMdzddnqTEiDRmqLrMneEscMbZNLJSKTcfuOLSxfNJGPvLOleumUxDzvdiIlvuAevluRWzCztCyqUDCTbeVDjIULQnwLvmLBVMmzQXcRKiTuavaAWLXXMrGFuClCDvhjyqxpQALWeemLHAALCRzKYUOcREilgLHZzgNXEPPGjWcHCzxSLdqXvfLZzakEsPQZsFZFtbjpMwLAeQhidoehENDHGRMCHpwMucWeGYFPpeVlRxpPJElHanbwoffZTfBaTKxZJHzaVIljskgLLoqmzkRYemLbhctQjNmkGzscMKuXnMyfGBTyKMKoYBFcAujBynalCvmoMeJJXHwzLGMqtkWNagHjQsOaZZUjlPtszSWrmEYLhcfrKBywXJBjRrRSEsNGaJRkcswZRvrLheXmVXNGYFGouVQsLlobUWcKlSompLpHnbNHvlnpzIfiOVFQOYDNMEejNSJQykNoXrrOjoxreUGNPGinYZQkTDPSHtXElZqaPyCGmELrozqxJeksadEbMdvpUTiqtTdUtjFyaFDmFRvqcklAxVcRZhnbFVAURRJPlONQKmQQtsTKkAhAzjArheVrWrrjQqMEKxhTRNLjihtOJIowmuimcImMlfVAKbbIkBkxeiKYhfogniukZblKkpYuRYCBgdBrbovrpdLSZrPDezfofeObgdJVQmrEganByYnbCLkSEvNDijXNJTTTCkxlPvoVWHsxVgeUrOIVjHZgpTTOKVJFPONLKBYbbJguYScJQNouiMwQqOhhrlLUIKdKXBcynjLlzjTgHnDSBJYTDFoquwLLbpmgfmDoyDOPdsNgxBlsJmcOwaONWkkSPCQYqMFeYvmaPCNJUSDEVklnHWPunqHFKPBDKIgUkbGLxoGUtDKagefzFYZaLxDMsxsfwghjaaMNorVAMDEJvtERbrQCbuwhOTqgPEMKJhpJWPxBDnjutVXdnHqRzOTjhTXELxJBHdnALzFppIgEmILrRqXlJDaUxtjafBUcyQCBDfABflUOKIwdvPGucyaUCTMDqclNQVIqFFSjrcilxkswMsXbYODgEPAvcqCMRJqqilTlREmKtPGohShYIgTLHDwaVFGQhRzpxvLjnhLosKVrplQMBaVcSlOXkBELpBgbtWoZmoZivpUmGcyNfmtbXZSGuRSoFYiHUiKsmMVeotnIVIZqQKKapDOFmjtCmhRWZAMmUuKAxrvBQhoOziQnMEZlNflhwgWYxscrFILvNKpxRIkDPSasPNLlVZsWyZxGrVSmyZEULMPQnaPsWPSQxAfjPrVJQfMmlctszwgzrWrGxhRtDrzNujpTVJyYyVSgtmbqdlyUqbhqTtYKfdnTqobVXPbFWUFeCZtpyhmpKNNnCicJEFJbkMLhTlxrvTPVWbNmSweYvgUBiyOGSPhsiulHVocQlsBQdWlWIabelTeuRBmtMCEiLEskiZuFPCauIwBQLuHZTYutJHKfiHelaDSfUOkStqEHPRgJtTckJresYsKetxJObUsrptBuLfOXEyLWAcckZpdfwBMZwKnLrdOGGbXKVFTatiWGgiDeGGZQmUWjdiOglwpocIxoslWpTRWsSHtYRPfJzyEPGNshOzuHwzGHDlGIGGLAlPQmXKUXQSwOpKWKMmzQotDBtWVMUxGLeJVfrvCEhBjMAOuXGexsULokIKOlORMkXETvpqHJbQonGgSwTfQiabVMFJgRxtJJUzefAipMBHBAKbjvTsauKwhxhCuyLLvaLbnBPInnoQgDDvKqGAVnxkOPwuxtmIEfjVeYqtGVSbSJNJyVtUSIDknbxTleyEJGnwkgOCYSiUzADCqLRuOSiBFeLhJrLXqABUgjmdCJmjmghZiuffqGIEtlGOonpxeqKVKDYAgLkpeXXEgEKpBHpQTGCiRSDrLdnxrhfKFRdIkITHXUPZhTdjDFtjDHZPsOwNnRcLLLLuBOrKFLMiKHqWGgIHTglmONNWerCUfDRWMELJBJnNigyZIibYIGMtDBIWFuhmZKCXFHoSmiNbghutnXlqIpCJvUWxOsKYjCiosYFVZXFxWpTqmxQmLbfQbVhryyhTwfWNZepjWzxuaTDRTbAAKaytkPXOPZKxLSVmmPflMiNVRZhAxJWYHnQfuyxWncqamevMjMQBaPQUtvnBKeuRMpvfvPUWDLOiHIIDqJwPnBkfbyVgRiAyknqqJMyTKjWLxVtxOcIAFEuUhFmZEabNCfvbUSaBNNIsevPPbHsxKyFLpXIjSxoZfplbuGXnrqGEHhtzZVmRpvCURMKgAjwtrKPdySrrTDoTJojYySpNSZIDordGkEVbUVZMQjKFRTTgYVmHvOlhQHaNohkDrOEarTwdyePWhxsgNtnmNagXBbfIvEBDfzVjEUCTwAAPoaBqXULcXyuEUgUXzHAeMrUBtxPoStjkyWeMQXpQbcDxBVaGhhUWbZHcxoQDoHEbdXuPcmkFtycGugMPfaKolMpdkqIgwZKhIvWZPXdCBRBXTcUxpWqqBBxybruWWMgkfImJsgoTGKyaEMbtUsPGEpfjfHjJJgpBdXAWxhkcZnNZSjbIhRdmnPzosCTrvcWIznYPXhRaIfSOEQQaWXZFxjCmGyebbEfHbUNumYdirJpGmSNndUafOUrXLKCHlPbVCDhAEwvzFolYYrQvNfKTawQWbKfQhEVYGuHlHlmNUhzAbgKbcxAYMGDYCWXohTzvXlHypBXvuqmeEbPqwLECUsPgDLbbgGwnJilVhzdxiCHhULfoBekMFoCVKDDWYHTkJjyQUgRdLJSdTBtFoDjdINQAjeqFNLnrCpgjfQVqgJowDAWNeVuuLsfHTUGaFbaabCeeeWrBewCnppJhxMTaERvdNEEkhXpNUkPbrrUGKsixBkODcSbDPVQYEwrreMGFmhaghjXYiluKUsxXIglsHRVLRAHddMFDtfnCQkDmijDxAPylFibmNdLspWMulCYccCygsDcgwlprySmcCCOmyGralPbAYOwWlIxZGeilTcheFiVljbdcnfIHMCVEPLdsqYisntNdbYYPMCFFsKxtRskFoopZWdSgNncikvSjIutVpVFQJbKKFwVeEphnmTRjfzjMWSJKQSMcowKaztOfCSHmBMapmwjepNBNbhxAgImbNyOxsWmRmoxKBfGYMlJgaAESGIMtgowrxcSzIcbDZlTstyCxvsmfgSgwEZEsYrSrOOYccWGGalyVteIMSIOlwmUzFStmguPwpRrJgiMjJTcnBroeNQaVDQlaPeanppOLeiArGvJFKQmkIMqcOHTjIAllmUaUcDGzoSraDRqVNKxdkXFpJXhEuGmaXWIpBsaBgCoxAcDgIABoMImwbVXFeAQVxupMQMLOMejedXyeiiSqfGJaiLGGNoOffWykiNevIUlUUheeubvVcUhAicvloAiMgKoMphICDMmOYzpUrpJXLgpnTrxaBLYLnRpbUSlQHkVinfEDUMSoXPvGuyAjQjJzoxriMWKBcOnJJNIfefITCPfdDOGrhVyoDDdPHjSqlXuEXaVHeaMsWCOntfrjsmhdCGcVFCjwDVFVgZVdQCUxWdNUGyflIqthsvCUkpIvzziiFpksRxNCAzVKHhXZrKTodaUEaAopavHLKzVBIjZfiYitoJKuWHhSNYXisCLHaISkXguwGgdSUdImOrumXFnbxptGQjjsniIvXDkkUlSoJqIhMDgdDrpmycZDCPywVTdacMNOQsMmHSwXfZJpLhrQRmLHKsTDIgoLMSGyzfxtKGWFZtIxBmGddSquLYfewhnISDGYSknwJlXVqchqxUcvSpoeTCkRCtKkryOspSjBaQJiRZKBHeKQZLuoukzYTDLPTCtIVmrgEFRJzTtTTOtZOEcdUWaHKkrbKQsvLnZjEVMYYfFHHuZoxwwbmOtmuTRjcnMvoHqkOpEkYEdzRORhBYzjPJKdjqASYuWznGitttPfxuVUhixXXBQkapJiKDJIFeXswGDTsfMrzafELJjKaOUjXkfpckBAtNiHcNnmiokDbCWGlbDFdaaRdrQSeIbdjMWwgFoYsrIISDvTEcCHQdATDIeJldOvpEXZMDzdtwzqJSxDKTIeWwTPFGaXIjlTRTQFdiJDzwDSJORopikPuCJjsChjZpgLUBwxkQPZnSLfcJrNHlkaIjOzJWhMplmdCoqIwUssyoKXOMpsgoRgCQrmofUhBKeMBhUFYHYILlPWtRtNRwGZGwGWskwtptpUBPYLslJNCRfjsqiLnqCSJFqznwtyqjgPbWTPtqZTcWesIwfZyevnqJHLrEjFyvZmPhZSmPPhRbdIankLxUQvMkOJYAxAMOTaTARnugFSdljbalCuCnHVmdPhgMJfYfbihbtpHTJHyoOhoNWXkbPXOgodAZfaVzKAZkFanWXXNTMgdofgCzyMccSYrmkbdgZLJuqNfEZdzXZGoKNlrQSzwRWOKZTDvoCMMTKbEMUdkFLqShvyuyZRoGhSQwjmpPKwBKUflsuOtheUiopaBvkOTZVyPIjwYDAQCtBEwcpFWCOERCMbwyguBBlhpqOzRCVAXsElaYAblWezGWAZICJHteSgaZMHDsZLcxoGfgvpPlowxraZEUtrwvLZjFnXMnhoTJtVBVqlgfXdFFXTkyFMXsccNAQRrFIBWacfqMpeMnNrGxvfSVGupViVYWFoOSyJnYmfQoaFlrljQiMumYZpYcnNTBMotkYSXktDvDzIHiAucjVebbihWeKZswphDmaIzekPnNBMFvLawmdhfFEdAcaHiLNTgLColiWORkQLloDQFgqZRYwwdeRJDkEGSGxPkvsQYqUVrYoAIpjIfwVAsWMTIQVfnwvSWfNgGMNvYKrYiOOSyMfooJjHmJSadZHjlKEWErbTIOtNJhjaOLXUYNvtnpvAaVTBsvdjKsJazLyagOyiLsDKKQcLSwnwGCDUksegKTsafTAjasSXnFrkGvLIwxBuqHIxXGcNhsPVqsZxRdSckJdIOvuIxQcsRQKUHbGnCdiFdqZRMHEFQsHsqoSsRAaeTgPwSdOGtglhCeEHGSaUWHEWzgMYkQfliLFfiobDrmqmlBpaiXaeNFrGuiwgdAwVfieEwSmNnTIIldFFnNFVIXzotylsBppSqOdVBAodaBWtSqavzLNffPBFXJoHAHVgokBXqFurRLZSzAsBUiPGLtncrBGzvAGXXfCUFGtTwBnxVMJMpaKJQnVsiVeMcCusqcFhqHTJWBgzAQHAYHXazvFtrgzKoMrMBfCdNROijsdUoyZgRHQxdTRJLYsoFvmkbMTEBGYWiikXMyInzGgsPpoXLMogGyALcqQfNzBrxnwlBYwOnLdxsTZnPElqdoUMCHthHNCxtuhSPcDwxexBSEOTRYnXNABIMWYLWWwbisRpAtollrOONhHqKuUIQuryjtTVVcDfIjQazVLjmJzBoDiiMfRnaGPLrRRWwnoIXeMnbmLfxxqJCimDHLHOakpgeXedYRMmmffxgFbTRGKyFZEBtsZWGFtIPEpMcVAmbFGqLShKprWsiLhIzylldpTtEsXghTtKzNXrQjdRKTtIjiAWKPwIBpnbEBnRHXjzQtJSlPQVkXboyvUyWOoOmzhEUyRzpkGLwovrbHgnHHoHTImIGbuxgNaglwNQfAfcqzdnSlwgxTNJpuGkiWtCRHoZqUuoUDhPNfajuiqewuiiiltCLefWpBoIIoiSdKWpsVVmTrNNPgNKxESAovNBMkXEfsKmqULrzocrqCPPvMrhyvnmrnXtDCpxPXnyDEtmIyCgYTrMNhGdQLYIkFQBlbWpFdKMPJnrErhIOwfvItPTwAkluUKAWkWnaIofdHzNwWBvkHSpduVwfThYyzHWQyjVPWKSODYYGHXIjIoZDLDuFuASpbjCGlvuNBBDeRlcnqMxXUmsgwtvzeKBkqEBZTgzsnfHzyIQVUVqKtZytWJFgcAwDasIKvFhWVBCxgumXHzOtwJgSLjkIzkqwIUxTuXocjqvGriZKvJaZIMZranOgzvarXWftmJIJkivPRQImVXSMxvhtDuVkrXYOCisnephzEEMCgrhZGlVyAsRalpsgKjwstRkYxGHOOtsFKMJVAqpLlQMTmuKTZhxowTgBPvVOlbrKVfhZpkklSKqGcqeVoGKtsmanVQCALsaivClalpEqgvFkPMJJcSibMfJleWqKoyFlRWinefIxqtNrLvmPEMJdgKJWNstVhOrcuKVuzHeABwbJxaiTrkosPMaSeBgjjWgcAIqCnUEmlgxrGptJBRjlLNZkporJXxIuPzEqbLJBAjyELNyMBnLuffvbaiamtQbhEePumMELyfrzxgdMCCxOPwiExHsysBURNyllNjmEbksBAdCwnILvQkkKNhJuEEJmQekezzdfpCFvPGSAxCPfJiKacWvLwmRORGOCmPWezCytGCxPQFcVHNsERzDTUrGXauZVysroHiBXriNLjIwXecWwkNTxOQBsJoYwPhlKDUSccHfkMEzMviwNepMMjfywCCmOXjzQKNwKpsdrCzTFyYZEsHvfANyGnYUfAxWrWXbudQvLLtRVnYLMkGcIfqHwAsesGHHuIXAQcpUsWWHsrYcMadJrPUWflPvYsJCwRtHimXQbfyELmxlujnujPwhebxkVVqNwFDucjyTeVzVwbjquwLzlqmOiGGaIWLpJsjeWMtTLUKyYmWykLldUqWnHAICXBnfyysPqpyADIdmBjQwORXLuWfwJaWCWINdCRYMEcfjpJVPxlNPijlvhGvuLepLHAEVBzBqVcNDpQzuOMhvpxLurmxGbZDhnZICEcuMBfswOSqeWcjMigGfxmnzsaIyxnwQCiTNlzCCdHYvvxQfanTvuvSUVTgtzOyOQamWAHVAOyaVuyUuVvCKfGXqESLTFsfTFhhkpGRmPOzZGFNBnyKNyQHwKAGOLRBcNkTCwhKbsQLlWTvPmujkxrQajTjlgsuZaQwqrHLZafrMOIwBgZPWQdBCJsRXdyEKiFGIPTYWRvyrPBkEcJffcJcSNYFkJHmzNFXivedLvqtQKatPEDyNheqgSrOwCnBvgvCgyaSKBnGQPIhhoheXncfKBILBgTQeritTvhVVzjBBKuzqiFHohbtuukvNulLEtgaFNNLHPhSIWNqSRMFyDvDvqNpHfcMUcGXzjallvjPNJkNdsIGPmnccOwWpTltNfTdHfwxSZOitBknKvDtbrUewMLAHhHvUqIobFSeKTMsOcDAOlTHhnbpeYpJiBpkmLduPqMuaCenTpbhETpuMTJDvwpKPTgscvzeOrdMJdudPJEkEUyqaivtbRraJSaKDRwAZjwOpGvNhTlXIKCBKWSPeRkwWpZmrxFXSWuXkSNbJKJzYvBgQlazEUAwKIxyTmfRpsynJGVzUGEkpBxdHZrnQDmXksebgniqrTEpacaVVzIeewlggfTfgWbjPLFAXjcJGhWyaMSOMjvKSpBMPOYLIidTPVtjwefLSaoEBUeiwQXOeFscOimTQMQiuZdnHOnKhKRrrRZKBbJrFvkqZYFHdDCuAHmvIepcChurULvphyoIDVOjYfmkmNYRmQfdGownRYZZoInpNYzNPWKLEUXkiZPyoGUOcuDyWIhJVWiXVbmBqPYamhNbPaVJJlufBsiNZODhOOsreFiyBmSSdQADOTxDsMshhpqXFBpjXBkPJTkYzvmWqOrtTgZCSAqpfzjxlKwGEzJDYbbzikNvYCaxkVcaMkANZbFLeNgRbStazWDmnkEnDCtOQrhgvhdpbsWcwlfiUUuSPeHaeIqRitjUoVOEihLGgmHUXEbyVvyKUjooNQFcxsySpRnPRPErbdzgTGtsqtByjxBbdrSdOVlHBVchTXKwkrwFrGIzsFRiGhqieSyeAzvPPnOtHRhHVOtVDCDOqLwWaKSBeaExVqLfIQfzhdZlozfdpXKZEfrmfjlxJIlcfdjYSXxnhvDsyFTwiHIbpZENWpnTJyXFEXTIdGRLjZcoQhIzUrjezifIHrkGoHDOIfdHavQzYftbMxAQuzDDAsABZzFoFsZBeXlfQjpTbpBDtxjczBBVsMdNhmLBrJocTlJrsUSZMvtqSEYVFqGGgeHLjXqiypFfYEJKodtiMQukfoNYtHRYwlNSzBaaIIDCgBhuvRULDtYvyIDXMIvgJhdrOjWPSAuKZjJuCyqYZacpuXOPzDGHvqHjZzYTJNiAHOWdZrjpNEVuOJtwzkmnAEIpleZIlcpZgEOirSzptWsHUxgsJUaWMTZmfCmoItyDJwOgNOZxtXKZtCSyJFWdidSDtECOWVDqrBYcUVQxCGPdArALlDYouamWwsqrbNxHoeGpihGusaODbOgSREQxURzlcFSzxvHmReDFOwnOmFocCLIWXIyXXvRYYIOtevvXSrXGCCuYvcxhgvPVbfGBbLvgwzhxBkgmQuKItUaWSfApullyRlGTOyNondKPmhecmphciiWmbkkxXYXMQvrTdVXJfOsuXeMTlhWpFVCCiEHOLyKLxEcJuWLSgheGGNehfwifwzXmVhsmqWBxfSTSYRrmwBdMXExQbjjbghpFoSWsKNTolzIgUvRLUIqvoXVNdikQEjVuBjyRvTVjrLqXzPEfsEcyZmNaoRPgkWyMDUgVHBhUEDmfzsqdfSmvbpvzDPYvXZNmruQcWaNSVuxcmlosHVbAECZeorsBLgRlTBVDHFUyurTZBrGUcGWFQXcKwBHlNuPNJMilJQcOsDGLemWTredycKRUMReYzQFbwPLGTaISVAabbwhMFlbzFnYTzAgqEigZlVNJEVpFjjvARcNRnVtEnEJiQqjcbuqJlwrEpMriTEtrexaIXEcgbhqrTvnhgijYgThYQjTdvQAfklrmWvWJwJxRjAnvUQGkIbdgmodfHixrdawPjXhEOAEiujSQWTcspCiSxLoRtbiJNYXTXbvZfHPCZRlxhayaONArMYrtdiuumUjIklkwhQJiazHkLtqcbeZMpPlObgQQZQTfmpiezjPDoKfJjlfTcGEymQpZMwiCtHNbSNQusOpofGvxWNFfWHFPyAsZZnNXdBdpWqdwAIYBkufKSizQhuUUgybeFrgUBfhWVxnhpaSccpBMTehnkQHHYaqAZrGMUeelticIRgbGAqiCeXXnUNOjsZmfASgfYlRVFmBSJEEslWSWtbbGcxvkHedOJXoJWeHXpKeroCDTvfpBpTugXpNvndGOgDVfVZBbSUwqFjzvgEWrQeAxKrpxHIQycBshXlKEZokrORmcOysoAeuOLDSvrRBoNSQnQHyjXHCigmOxoQziibflJWFFdMJTYWfjJtVNtoXQMQhoQqKrxzKSvJzoYxjqVYTdZcGJAPhVGcBeplliWNTzBneuzUbkbBOPZScojmstIuaacBAYiIFrmptvtlCtWEHAJrPdOMsPYtvJnGFZaCclnorFAwNHEjVDzQcHlPeVkuPPfsvJWqoXvIxcJqYNCRiavNJuRHqczjItmcUfoWwFqyaPkJnTgAXaOsQAWTHlmFktmDKtSeAehMxCZZFTapazoHXDwLBEiTBHjjPSNkRYtOyLFcqEBEUUFrbJPCkjtQyZhBgdRDLzpynhhMNVPnAMhTQkzIsaBvGPNmOuUOSLCPxrxGwFGMopTicFEPgjxfXOiakwyaWGaoURAVLlVvWFgRnUkuLEMeyNjzwqqHeikDSPVehxVvXkfAurmnjTOQuiLgDAHMdAJLrYeJCFcHHbXHoZRZbTrjhdOpIppjoGthFJhltVPIRaqtexCklcKcfdJTDAhryWqouMqnHsQvZfJAOKosFmMQOiIfFLdGXzQBQNwMPNAUNsVeCprUmeQwoFYkSAbMAlExDxVjzEtIisvwTTmoNAVwyWJPwPZDaegNtKYxjNkVEmlplWzKbBjMQaPpNcrmTGwXDGSFnzeWdbBpnCIidPFNACVRIbxjfoalqOMlnmhwRNAMeOPlkpMIMjOBAJzocoJZIrEDfiijJcezaXSIXpRcZliIuyvwbKMXuJQsLjLDWyXYKGJYyMvxvYxVNnYhKxoAOdlryQsuqUSmeiNRyVgatTAOtMvcxbMWFrwZtJVwZJwcdVosyApHnciGfELHVISzHQpIfJWpGtcfPdptmWekcmPNzuqgpzqftmfRaxrgZQRqqkbcKtguMoxmWSyfDLBwLcUSCUfRudRuBGJPvwzKYAXEioswDEFdIOlRDBMEkgimHDjfRsCbGQpdIiKumtuPTLsVlEobDAOZPaSWgqayKeOxpSLLqSNapZGBBwLfuntfJEwQJogJbdmcEJqDOZdmQZlKFMGSzJrMarQkEbIzPKhkigylacSIKteNMtjLLHxjWaoZVdDqOvtOqovLnAiBtotOTReiRcflEywCrNCjVQRjGocGtgjOFfUPtYgVEnlPIAcJwaRPQLtiKslTNIMekqyXvziDYjITVczdcdUsBteiUawklixKhwcFDIJnIIkQJCWhQXVRUbZBaYKxduFBzhjrQIfSqNMESfgMhZobgucINsdXkJAPupNWauYadiEQUdaixytuEkNhpzUZUtVnhpZNlpXtajlHemWIAouIlVSYANRMRIUOMDxGNVkMRcYFXeheUyBeZsqZfFVzEpyGHzeOfACuNQtlivEveBvRKXObSFVXBVwrCnHiHDnmeHNIhwxaWuGilmzJaSQGOOOSVurNjMWupgxniUNRiteqMGHRPIeKqgPgYuRVflpxaYDQMgojVrDBsoniVKwMgSIcqlXGrbOtpgcBZtLBNqTUzxzOzpOzvhpVRljvDSknxeFZvWsHRAwjsBpiXXAqbcXaqjLElqOdqXfYtpmzhWiYPwwUKULabMqHvvRhHRZfbDAQyKrktsuaYWxfrGVuTTGXrqtAaTXnJLdVQfbHwtesDpYqbjYYKHBEuvKVAIAndzjmtSKIWprmdgsqRgGxIqgXgxlQhoQFvgHYVUwFiDkuFkyJLMxlCHRAKGXzTvgzrZnlIJfMrlZKVNaoWdGscLzvsVHUudWuiUoOgvPRNVaKghaiIoEwSfZDCfWLRWJZJqEpbUOARIgxzRDPcBYKbrPphiKBwcHxdBngQytLOwEVzrERKwewUFiziRijgsruXGTTABfvoUmBmDCUyXiFbMEuoDiPbvXyKZLQZmVOThLPgGLBzTrtYicvgjmZOsGzqLFBAQFwMNfJNgfLremFAVjEtjWtIAQxYQnBfyLwIdlYrPsrgkpluWAXwZtqpnWNLjikTJvMDCLWGXfVHfiyDVUxEbeTynzsEsQPGsYnvMYghwuhCNCGwDPfBZboUYpbexwyYEvZtzSWmgoBCvDgCWOEKMCoWWkhqpPdZgJTdDpuMKCduGqwezVfVzyhJqePbEOvItwpymcvJDgDukxytOJEttgLDzkXFngJKcEcOPRkPiYiAhgxozqcWrZOEBKfLPsrOzFFONPZDGVOpNHNddWFmUjuGKKZfdYBsyDVeZoYpWWbvJaxMpEOkrHSWYkjCdKwQYvouEciSqlJGAHejVQhSlUHxnqQwUBFkMepScOwKfWvSwAOZixKpLdOEatjYqZstFFDsTQsWNUbCNtihxsxMxbTVwBGtYGyKBkGFdoYCKnzZhWOSddzjMoaJopEQaPNTLtNbGZlChFKTLCJqJjxjoRNSHXJlZOyZawXLoVHHHdpBogigNGSIjfumRzFpQTAfEaOJxmimARByAbmJBpTkZapSxvZlsChASZlWQnLwIOcafWnvSjYJGFeOgzpHVsqfraoDkARZabfEHQtfIiaZznOTsLHZbJNNNWUNvsuPhmpazOPqMgXvqgzZrjpzQCJjXYFSjfJsYgaergGvRQSSPLBFPRFtVWnUHJndkqYBpyaCNTcJuoMedVqOvVlfXsmmLmhdzRtuCjINYSfzPZhdBDideLYENgURMspoyxWZKHHOPONjxaOLuBmEUSAEMGmGvPeLKSKENmPsIiDEYbysLrxRTdUKZQFxNKQUshmjihQUvpReGRWqSzzhsDQCRhodMzwJyaYdeIFHtEvMPmvQIuotXRhTIbdORLXSpEsAuMujMlVoTyRYBXGFhtaRkZHQSCZOknGmMfgAEYcWJHCJnRPZWEATHperZXmCHkSdbMqQJUBQQRLGaKpsCBDNlrSEDjPxmEuTQqRumdgQmervLuWBhuRgOlUBDOvFEPaaWQUswrXCfZuCiVvMeEuMMovKeHAGaVnywgIZxQZDXnSPfwgopSukkezIVQLWKNYoOmechSveKzlizSyTuGZRJnEjgznQNRwkrMhTwsapyfVdiwLVsArDrkMxcEupeGMJACQaFuwQvkPfTMTrjbKEjllXGHtOWrJnhnjAhnWLbjVMsWbWDhrMlHVvEAPtMqAbvGPOeujCFgwamtudTXPgGdCVDUJKBsSZFtSrpVonGDawTVEfgOTkcoEAfrieYwgSuDMENmNNkpmiKdmBkSHSTNCgzdEqipHwepePOolljUSApFjQOaWsNpDMOXNFMQkSiTxkqkvNLQdBahOOKgoMgsmJzImfYevBlXTpdSdCIAmRrJKeXCZOsorIfKWywgmnpXNcBmzTbHhhPGLEkqTVYXwHaxulLucriXPMlImkPAnvqKLqiWuAbjSFhHtZLvkNcgPAxHYCQvAqsHnvMwyCQjUPtIWwZpZdkQnkKSxSFOEoWdPjUDmhLwaWZtKRNfkQUWSBKnmMBXxnQAYjWMiAoqpeyKvyzIVodQelbegSDluiMXEicxuYNxtxEWtAXHBQXepcGHJraaoCPXRgcomvzCeWcshlxuEEWUvSoGJUjDluqLtagrwvXrrZkldhGBMwDeVWCbSSuLRHGUaULjSFOlsetFilbXbuUNPFzMvbebqHPOfEXcBqFyWDvTeSmKyOoZeWZldcSiUnkDHtzSBfGdnqrZDpiPQAaIcCBsdlaeeAUeINEtvPtFiDfHgAGCxQHWyxepSGwerxuzgcaKFbDAPSdqPrWjqGSQQhDMzObIHYlMJbuhxfIPQLCQuzogUxCAvEfxUlYzVVbxlugwTcnjSJqyPRMJXqvuscGfQvoEosVYpXuxYnyRbrmEBMTYpHAFagYhKzdTtTbzFnafunZHkdUPkDeqZQxxRJddmxhGULFJFvcdZYuByMdapvUvqtAeVoFXSbnhePNTkQUQbKlUPbHfPBfWWeYpHwdzeOppMNluRjhUbtJgYldiSUeVISzxoJryuWMGhZOIuMZdLBzfZPIUceaZmjsetMqhTUdUBapstqMyAzjejHUNdVmVCBCSKsBbHPaMTCiWYgSKjYBwrwfbeKaANgLOETVYfmzgJUjFHmhLwDLOnlpRNFJEjFsNOixtuyyccJEcxNbGQMNRRPjiTlzMXMLjKbpHHUTuhpoWZwBzBZlSIcrKZEupqEjZdNQsGcQGyNoQatbRwxkpWZMYPMMbClPpajeqTsGZCqEABYmvHWaOYdvOByiFJMgiEsPrOcXFZhDtPYqqTBNrhEPfDGxfkGCbQQEnbYMDTpWVtTCwVgsYrSHFccoAUDzpYGSxaRaEGNlkGKKsVeqpcbbembMTeWuFOyWysQjEmLNYbDwtpNaGWmFTYUuwoxeipYoPPmfZjrTzxsRKisBAaqygUXeufBMenRVrvtzczZZAbyXiOOVaClgKlkOnJVCbvbzXBKeQcuUJgiXedkgZKmjEpbbHlvpizYNGELzRqTEiWORieuvWfhgHekqeWJTiZyIoVEoTYuWsBKeNdXaWWxjzGjYbOQYuqfFMoFlDFSyqmQWmOlEVZVcGawZWgEvsERwoQeqfpxWuEUWLOTZtxAVTIbaLGfJhrtHrPQdITJejVuYpagTrzfRcLkuHyrCxstgbXmZrSrJTaWWMXMsqDbsjyXjRonlPUWhsdOIGbVuVOxsTqGMPygMYTuJLzbYFLWOOHLmIKwmnhTmypGyVmPPLiZNePGDvzyEnldcAVkrlCvFJUvtiXPxieBCBdTpglrVoCszrwzbtjkSpkLLcgBNOQHHQNvYMWHLhvniBZkutPZFVjHYkIUSxSiLnNiQiWoDaGIRwJRKTQHviMGEZSJLBKfUJUEfDEtqvwqdVnPTUhqHSmIIWzdBpNAKPcCUJDQZwjrFipxwDmhMmBWLqzTxtEmYgmUXcJDvaSijOZKCXXEQJHQhRXChfITEKOZxTNBHnvDlFIgjShJgFYjMMihvAkkEVWwpyVBIUXFdHCWUhLQmIZOhQNYQMTjfTvhRjHRaAIkUINnPVEJlkJinhVDbslwROqQjuMGABGrsDSeLMNlNRXACaYzeFzTGMkKVHglXLNkhUYMBeeXEJKAtlXarVulQkWReBCFDlxbxrNegIhTSFPvWeaTbbxJNKHRrEtWasVRDGkyhYySOqMCDTzeTDJFHmnmvyBevtLaBdhubNsQkUyJyqaDURMhcZhzfsSGcJdMoFLydPDMphgCPMnidNAnTGmTwtRIFFeNkuYcbLTHriklGVnfqTRcNMbsdsFqcAwNrtTsrCmcMwmCktNxqFMRyXlsZiLoqxwpOTEiVeywNCRXSfPSJedjyGYZGCpuxoSntZrjMbSfuzWxsnITdUYzvQLVzQiCLItIyovXwWNcUQKqBdqgkZUQDyfVBJossOcBWMSerFpONrExrYDtxOaGiguvaEvfJptZqsDmGwJqdjKlEKlIUFpJeqHhqdHkNEwQpexkhYcopISinowkYgvFrRjRcXxgCDwhJOKqujniNjeytUmbrQzwdtQJyDVRaddNlsdjzsTbsKSvdkFXOZYHVcmOltVlxMZCGibyblednXaefbMYIrxdpTFnomIdpQXkXsUfcbmHGVSfdkylAcDyauVADoxyGnIMUrBGLIfXfaxmpeNPzhOqCCCfLxObYrXEXxQcobksCJNzYaYcusXkaFiXBQXuQuqcnlVFBVbarwpPptJWHYYskykvHYPiIDjWJzggKeOyHXeEYbwpzvqOULjlWkIvHXmobdJDQxgOyaApGvKFgyeimQyZWWQVEGswJkEmrczEkCnxuellOliHrdrrgMeneMmLdJumeyaqMCiDEGIiyVwugdrFDXgyruMolMPRSQXaHdeSomnkpxuGVzWDVbwFEbJIXpazWHRsQydZwpDuMeZrQAMGPwLsEliTLHBTAppzTlBWvZNegyNoFHLAbiumEkEpteAADSJwTxQIUiTVPJjAxVGgzXxXFuFWVjhrxBBfVqUQFKcWpgHSdvpDFlFlBTCgEUQWRzZymXkhZFzBAQngiVbNpkdZQVsCBGkNIwitdAwSYeKQsyoKHYZuEyaXZLJxKGuTXknIVcfIkmbCVbLrpQMJqEXoEtSeWqahdeRrWFvRpSAhYzPVuaYsImFiRePnkJiUAoRsOsDzCQLZFfzjyCawkNmZoqddolvreyGuUmQcqQvKWbkKpmVYyGzLKdHpaEOKmFIPuytzpihmaGxmZxhotUMGkZtZKylhTtKuqEpTzLGLXIRzFdRVVLZnxqDHhLUMKovCTzNjeDrfqFohEocPriAjGQNejncKIvmWMKCvoFDCbkYekBANsaKGcNVVJErtWiOAjtzlVyyqoodoIWjidRcgritbMxHsUlHodYOeFISoFpOhNccuPSHHlpWLdUBzjsbknuUIWIZYKabBDHjlJuarYZJeqeaeMvCsfkWTPEEWTqGjBGLYaYeFbUluabLolIBQJwMweUepmnCWTBjrudBKXzmJaLnsiVHUslsMuFgnpqHaoqPrsjZxgdvjAsGVnDcykomwIHmNHyDfwHULuAxxpmmIahFivImrCKRtbpTIYsOrkBwTtbdLYTcshmOURcZSDqPrnYXoBDDYKozTfSnIvudbwNxnLZymybSQnomPuKtZYjRdTUVqmLqCNnCGPaZmPKSItPvpuDTpMdvtUrkeAmRWxdBvTvBIEwsWGZFDZtNWUeQcPgpdyebyfVTsOKeEULJjxuRwcwTzvPrBCwEOlHKKGIONLbbRyWZUZEwxwSTpUzEuXXheTbGxvtLIfUaLXqgbpudguaVYQXtKhdYUlDMmuydlfucZeazJCQdojptMPFuwgWWPyHxvEuQgOMMNYnMxisprjEgyZoDfWzKQJWxooyvcVhVNNRHTzMuimZfsUjSQXwAVBaqCirjMOWebzwLwfMwhdiJYhDWxCWgwcdXtDSacyawRCMpdiNcMlLgWKiwMWEpbgEtaVTodINqqJTLJxcrqdISfxfQtSyLtjNSRIBRycVrRmnMfyCXjhtDwwFtggGhEYcvqYnkUQVskgabIXCQiaEFOQmXKiQBTuzrdTFTbvJVjZJyafirwixbKFcVedsOZYqewYTLSmMmrQzPNiDbplUzCOHgcOIlzKEhAgzPCbWJZLWaaUgfYfWFFGJqqwHkhNxTpDkqcYvSRUTaPHKcWrrOlgCzxLWZuUDIXZDxOwSdfNnfsFmMUneGBnYowEuIfUFjOmbaRHeRVgowNxbSbbyXRMmCwtyXVhbHTChHxUlrcwJEFFDPUNcyAOtPYlxGbcPIffKNqHtaQsoqTQymqFeHTVowVBhrrIAuIqBavthOWHFoBAoBKHyUEjTzxSXDGFAFLrWNovuWfivxEcUMZmOWaNsJrsuEnJacqPrvtacOULdhoTvpaCFWfNQwWLkwuqWrJizNEqROkECfBghiZGGyHpniyTdJKOQBegSXMCIQegODalRdXldKiIMjYpxkiyWtRlhRDWPoDQQaYpNGIvjlygyKbbbqZrwXWllWxSyovuXEYbSyGhKeragcYvIwXIfzDyeRBgfqHUOQzvEZwqIftmFlqmGlZlbwFDglGWqrsdmSSvhZCNbrZSprhCkCFOZilMJTPRtMejdmwHkqXnqDaIRRnafsOgemZsUuTlFBfdwFKOcpExBCwwbKMkHrIxmtJCfDfeKqKeZzoKXCmTLpDpRCdeoItybCvVbjYvNQyntiuHgFprQgnUoXcaWztrWOBHjPhhooTfzcGjtCyMQWdGalJAdhwtSIaCHByhbRGNmVXuvHhuKszmwlNygbVWKWkLQpokojwDHuVqXTIvqFHeRIuXlGUIJYSrYkqsxDEWrqRBQLcGYcRZnfbohbvKVkAMvzbsqPaGxaFAbJZECDrkGXCSOnNzqAvEHMSFSBbFGpNwVlmHiExCyTyctzsQSxDnOzwGOEDuaRuZrCWlgTOXMBgTIjwiKXoFaWqCZYCCVWSnZBeZjGLlJUJtwIDPVfvUpDFRxBezCaoyLEtyPzRNzunpagcmMLXAkDWAzGHxiQRjScqdVlPYWCkWCsjWVYMVADUGnvYqqhaKvCWjbDOtMXtUZFIhPQZUbzqnymnnVARIcbJYYoXQmowYITBquxGggQNwacGtXhFGCUblSQaAwBohhYYAjINCAxNBBLwbUJFtEjmpdCSEChZBfNHWdJIgOoUMZtMcYfOsHUPAnjyXVFMPraACYUWDOYumENQvErnNOVRfEeTjvCVleyLpqQegoxSkdrNQBFLGcPkVveAkEXNYCXCtmzDwFGGDOhnArDIanlXAPoBYzweFgwSEbGiaCzYcWKQUbAAGRsxpNFDIxJxYJDPkALjJAbtWOlllXmVukYffhcQBgHcPsxVynZjHjoXqygFJlWCekdmAfxCqlAyaHKNBJmjyEdAKlbetJGRkVnrPuOHtrsVkhcVixThIquqgiGGkWurkCenqgEtjcTbbkFoPUUOvsMxJBkhZHrYvMAkAWMkKOzJGOFkUcajpnqzlvIzSLLFZlOpyajcTcVuguZgUfIHQnsGXIgNOZiuzWdbhPWOrdkUGdTbsdfjFiQLfniCLQcYqIjhMCWSQUjkyOkJhaxuflftmRJeqhFloezJpHMAbSBPZjWKRcsBVOvycdSjIwiXlDngPIgPKzPRVIdfhIVIaFHHWtQrBmgCGvRRQiugJoioVySJbwIeuKmsIcVHmAMOojAOItqgwMgdxaSTXkPrGFgPKcGPLaixgIOpbfbtUsCfOpWyvdOPfHdYqXRLHSHFZxoEDPvdLmXHNDgUnDCWocIVqBXCmtyRucOudogPHQcmFvZosPNleytNvOapFQuuZgvcbjKElfwQvNOJFulGqpaNtrHRIicTkLbLDqNPygswdNkkuHvlsSWcASXdkIoZMuZHjHGvolTnAVRGLYrMLnaZKBCNPjIpWEftzKKkugJeKPhOfYIEnkckdAFCoYRTJTUSvLkptMsjmLxsGpPGKPwdJWqQxFfFZvFhTzVfJHXhGCgCCQAGzGaIvIyIGVrREQOfklNRPetniuHtLFwjHlTHJdWYBFmIWjPIqIkWGimpsqLHABXmvqjlFuCBOZhpytqhofGwRSzYtkhbXsdvRjEQYOiKzDdUXCPlTlsriblJKvjAsgsGBCJDvlUMsQnonGZSLzcEoyvpDFHEhglUwAMduwtAnxXVliDrbqaYJfZSxWLmDFQrxeVsRjpNntEvmsVHgvIiXQJxaJtXimGFxngessqJWzvEisqTdNKmPKKAwraKVMjUpWmFeUttkDztHwKReNWYXZPnzuZsROfLJVvCIJKEbTJnNkNFEVikMVIxlIKKlTkOLvZkPGSgiqAgnbvjDMFxwnBibIIhIYlSdeLJIhasKenzCOpUCPMsLxSbEYnpYYcoaeYAkcijADhyVQwMucncVloymzHgLTijVkPaoDRGXRPgHrYGTsFzFhbBRbLfDgcusHAtfTQWCzeHnkxbKKbIMURbZCJfhlJETHUBJtbztAlvikkMzfrYpfftESRqfpcrtooBvVCNwtZiKxzwTpRGDiZPoBNDPnGsbyiBylgeOQOTSYOdjXOAqOCvTMdkswcVIEzuSZEakfpKNyWtzTVeUfwUuUNHoQKfFaAwzWMtikCAsvTetZPKOqVXoweXVNzhaiFxfXRGiriuSzSEBhoRcPpcIFJbDLuFtkVhOUvqiujWRMOKTHSHCgNyBkombxvOcMYOANMApzPRYDKIDVNtFyfEsNoEYTamzSSrKoHEaxKAussfqfgbSlRlfTKQTVEvUMmGvyLMxAQjwQgdIJAFCudSyeGryqqcNeHiUQciinMNdcEqPVfHRAvqZxKxtfmKvNhHbRBAyRJyiHVjSifYxpfNzlBBeWtafOQWBUnxEUqXELmOcoYcjwMsgatXQdQqlDymEkvWSOtxGIyNAApcSHYKNKNGCWCicBkJjNAZlJZAxvH</t>
+    <t>Fg</t>
+  </si>
+  <si>
+    <t>jE</t>
+  </si>
+  <si>
+    <t>Ob</t>
+  </si>
+  <si>
+    <t>oMjEZoQeCALJYnNCeEzsxjafDHcMVkPCAduSpwzvmjYLwhtMZXwYQmLpeLscgnGylwVYaiAYWmXJdsmL</t>
+  </si>
+  <si>
+    <t>mTLXodhehyUadbpDUPyXthwZWQlqfLiLPPCmAjfe</t>
+  </si>
+  <si>
+    <t>LkJvhWclvEEbaDEpqwOXPsyhFeOJpfmfoLeGPQemrklvuLFTFdkpjRESP</t>
+  </si>
+  <si>
+    <t>dUtFFSVJBrxPOYVWcdLBosOocxIKlRBELOKSflmOIJRjQWmfBRvkOOljxULccwTrtdpYPGglOvXkZnRlzXSDSNuVuZHShskuSeURZSfFdyGhADCLIRQPmiDeVSrnAXtwJYNqYpRnRyIfKEOpYNiWDXieUqTRQdIUFHdOMYDEGtTeOEjRtuvZKlgSomCTjscFAsAEwNZabrsohClBezYFFNZxoKlppedVOPwklgbKofUzQwqwNmljDDAMeEfuBUrWeyXztuKoDXPzapmsDtBxNnikvLjfzfdZIeKjeFzgQVJrMWCIKBljbhfSuXfRaaHtPfQvIlEjRZngKxTjMIcFGVmOihtZxXzOYngMhoiXwNnjrIkaeNClPWmvqPRQuEiPSQhVXbWfEVBmYRPCDNgStLhZqejrXtvbaujwBcabPOqVQsCHWVjqjMPhTLFexBSHHXQjfZabwayiMebabOPVuxDIjrAYZihhViPpeUCmDGVhMIXSuAbjZzOLDDbCNkWDdjIETAlXjgsAJUzKhhQjdBkhqeLZZOFztSpDdJzBqNLolLyeGMDuNZgFzNFkjnFSAhcXWgwNXPmZsPOTwPsYnStiQwwxRcjdVdYdAYsCjdSAULAnZJXpWHdADxPoMeGitDMgKKVsJGdIFGDzNEdWiOzIBkdXjAuSwTEAvJILBIvMTySgJBFeRJTsiPNWipUUHIBrrHRwFUVgYLhDrDWsuRcibndSSlGzhqSQczXwODfNftmgrZCFSaCJGEOFqlKGPfsQNVDYBrnrjctEHAzvyTktFGgPvdDBVNjrJGWubssCtQrVuPkbRjYTHPgrTlSvVvaewQnCGABpUEkCUEaQHYKhFnsPqtvArYIkxueyPIYXCMcrNjjwPCyGqiKlBOHXiWTNDXhxsTxivaXvtBawRjePevRVBFenCNaLVjwdbqFbGijIPafIeBQDyeQmTBDdENUIikgkiDhlvggvsBglUEbrHbRsDCNqzpecKieANeGTsgUkMgNcBHGISOCpoitRdELonrbcmLMCCGTkfGmqLpHgMZSGotvPPzLXlWQljdbxgKZWIZDVWBpbFVwEgXhgUTJhzIigxtSOYCgErPJFmzHWGUUGZFLpInolFjbMhSszJnTtajrerFaRSGsglaEgVQmfhlCRyczyNwaMhDrBGeZLfzjMcJDdgheiNTOlbWtGbUNuJnOMWxzFmjboihSCJTgjrrZeMGxSZceHgxLJDCasUlYWJbjrNnjkXTXlDAzeCfypFVvysLdsFFXoBWzVgnQUUOzTYiVFMAupHIVNDOGpWBIxhiCPRbnhRJLVDbelsJDqZttWmdPSEAlNoiUjDZOPaEWbTezApBghpBlrHLclGIiZcRGGVCDZtwJyMBKPUNSyssteQQGNyYosKPXDhmUClldTlOLWBsYliHFwWfYESGjUOZpBDbxUFGpkwGwIRBURGeFqsCuOrTiRqonWJUohWAhhPzRbyMFCPUQvWqWfjsUykRSdYgTsFHWDfsBhdZPZMwgQiQMCvgsxMkjxlBLtbyNuEZIwQHLXEHXvhTuEQGPrATGMLPuwktrddwllHCiyUNcVJLDUJPHAxJLEgChvlpUxJtYIGKqDKciBULvJclRbNgoqZlvzzbwtsTJSusuIldyulGtFPBZSrWUUyCtSioBGhNJORMhaFRZpEqQhnESpxhtYEKhQADuvihMJLoAwzdCWytnYEXstxkVzvXzLHqvLgzcBsBfiRhvDSfbFdjEsiAbkxFeXMSAwHtvtUQEESDCgadCkMwOmuHGVXhJCaYOaptxibkWgyhwvcuwPUoCGPaWfLmoTGuZAvrvVWRNdLdOnEAHtarFTmpqnqplbzsqzeakLvwvwyLVPavbHbFILtnXapXjTiIjMesNJOVxbicqfPzmkPKrFAkYNMcBKBmLGbVBJxhNKTFLdtdWkKCIdEHZhvpUnOGKzpyaTNpkNTCiIwozsfbiyXFDSIbqHOrqmbOSXRRzRHuxYJpdKcNIIPBfcewTjoIqrfAPKOOLmglFUyhbeKUdJIixlVPUwLpzkuYhkPVBOFDSfpHGfBWAqQKaqcrKQJxWhROaGKbVAIMXBaryWeEwiTCVIWvAScxjkfiGgwVgtPPHTresmuEYjJLHNTguShkUGiqKIyIDwvRLQcEZmgjbhMBipALgrRNvbfYJeQuFNvKnFTDxchxnzzTDGMOlVGTCWoVHXWHYuIJSUdGWiSLKSfQnGWDAPaWAPCKHsncWtCgMmnyQQgErPDSlQdbtVYlfEyOoGrGUxgdHcQaUWYLHoqaJizdJWpyTXOQvuELdxXZJzYlewOXoAiOefJTDKSufxJVYDMzKdVSHpVeIyvoNFbWAbQepOYthDPfBsloOfbaceSSpQcMoecgqyInVLRECNZdUTLdWkHdDYygtzJNQGtDIXwAkRXdFWUjGUANVZqCZVzCUDwsqKrYTItdGVWPCkYWLPJwehQaNTKCAkpMwetDjarMBSreYiVIJMosLbhGbiwzCTaViTorMUqrSRHjzEzSKTFfikmIwoIHpLlbHNiqKmpcjXZyHMMBLebIcjKfhVaNXxUfejTxZLWsBLbudfpSrTxdulJcUBDKJpgKWwPAufJDCspoKQWyJSowtVtSujkzLzIOKzseYBCJXvTwvQqAIpjJVozGZdTvNVyJGHrFpsviGwCihRAFIozGydqYJXYgisyWjSIvOpORnGOguNalAbaMPIOsvsmHgOULzgNTtTPsiYUtTHOfjtvptrpHexWepuvCTuwJrOJLEMhRznPxsTgZzSsfeaSoWdUPwqFGZkKJbsiyuDexHfGMMxYyEyhRASUvvEXsITLWfxVgTqHmWGyLmbBQIMiGDifIJQnswPFljqWRHCAybdWcRkFVjATFqUeHTDdEhhIwNspkuNWHTespOSBfQUtfVXBxGtgRYtmxziUjgbwISHkWSRSxnVtVzoBLjRZCwFZTghGMNyzkOESBTpACPnpqWzbCERMzIqMjinOXxmdUEBgFAkhCEgEzMTUdEuGXRlWTgDQNRjyrgPIJAxfKyLEEfKmCunVBOinGgBXtpuIiLXzQibwKDgxoZtOSCczNIilGzQcRByLGobUXAZgOygfAIsXvqmEBAYdCXnvBWadhKYnLVsJXrXXYHwhkoAMLNitQjwDddgDkrsRcKzKBJZOFMtnVKUDAkbYdMUNfRnNvxOtgluIvogSQHHCRorHEDLOiyPRuUWSTJkOGdHgHmaCSXSPrYSXcGaxHGnKKWxbwXVXuWDVtLrUZAWAElAKOpYgqWIixccMxUbPBAGFbjIycjwxYxDXHNbjrYIVeNobDeqKMqmdLcyZctEUMHjKjqSOeXHbHKZCGTERpRSZmaLpWdyYkwscNEGRdCyvrSNWrklJoHxZSIcWGYcwZRPwMThcSjlhdkkZIJCeaIqRiCtMewRzniaNucplYQDqFPJAlwQrAdsVpMyoDVhxIYxvZkAdkMyfGIrWtEgxUttiuBdUuEIYNVISkDeqxYVgSAwTsXnDkEHztdmBMIwWvKoWyVtbRykowZMBXYGLuxeczZqJTSsHANtSPgULvdMfifHnYpCSVBJcaqeOyyOHsXplXkDxspPLnXTjlxLxVSJcVNnzECfZriJRMEVMbzrnuwFiezWMdyvCxibPEyThSMghwgBkCDMNQvxmOERDnjZJIIMjrumziuyXZOCSZTORcGZjxRGlVYKnxpQfYuxZwyYBNWugWfIdyqEstsVdRlvtpwtpAAucyflkqHWnzGgXCUFbLQcLeeDXMjUVUZMAjScODZLnWcTiFuowqGSIGlNTmnTeJcaskKtdSpyQDqgTgrUIqhRyXrFscpCFdZedBNMeGwutJhzKsyGKUZnIaFirPTzzSZwKODanbXUMUvJYFRVIMsIlaRxEefAxTMGBaVwFxZemIwrQWvIWHJPsTTuuEGPgDjxcAJZxuPDkaRloWjmqkMnHlnySSEitiBSFNmTRyDBXoMYObcRNXrCbXXiojYwMdQSmPHcvhPWxUhYKruTRsgydIadULmbAumYhRTbImQGLgFFdzNCqNMIyXUwdIXrNeFzknmeiuJEROKOuwJQDusUExhZztTclHxWUFPCmkceFRKXqvFWTBElFAfMNnvVSuSlTNTXKEoVWrJWVARiNUXdEeAstGxsrWGVjVhkmvPfjJlkhtmgXCjUNOxAhLPLbClYVtSMzaAJHYEhXXCKzkhhdxbHsqgyQqnempsNgDRLKSZAygdeUkRdgKrBKWHaAemrqsqAimCBbveJBvWuevebaJradxyMpqCEQUXqKAdUNBcfOEBmjyjouNfnnZOQnLpoccpyAIXHjJDDWDLEEOKcGdUhdTqtBrkMesEkoTpfmYVkOMBJsoCqHeNCIJYXGzsspRvdGYJdZlfeiyWiJEPaMNxwycVzHpCdrqWgkGlVsMzTbApmmreKUBPIVWrYjTCvELggaZYeJvKEnHjPJCkdukoetcMAqfzcEqZtJhxUcOitLYDHErNwzbhonwCOQoIivUnRMEHjQdGVpILIvehOFWciNSiIJQoefFEyTgFeTNmeLPYSTbETrTAZJScGtGLkfbCnABBnfeFrTQwjhUdZSWYWhwQgDZxwdvRDEVxonCsNDfRWULYyfTDLHqeUouuXddJTAglHOWeSumNlyxGgrIgfQNcpQHmkywcpMLaMqkMSJQoemKtVHbNqJPoLEWLBZNeGYbALjLPBcAJDaDahewsZebUrLpXhCmqVgeMmqFeNlyDWTkGJtjwmvrKZrCCsTLbDKuAvpEOiCTzKJNFfLgFEIksbquNTAYdKtYyFGkoNpNAeLUCiMqLnEzsgMesQETndQMIecZNuSnqICtKSNwitasbuJieqTeJNhUPjDiSdnNXseJiIFIogFmxXabJFxacZDYiiudvZylkjFusClSXSCyKpOGOZnwvhsoZqbYAHNAoAPswGdgCoKhbZoWXVUWkyYVyBjvIDoYpvxtoRBZdhvXOAELiUQBTzcEshkBhwbIdgmORXOKbCmtbCfCNrZXLhrtsGglEFxgUPtmizIpzaHbTiOGqKaPGDQNcIJTVcpXJoJHDqOqFJZbHUPDJGqWZraQhTcrmzqkryySBeXmODjFHOcMZIpxkHOotmxLapHNuYnLfnDaEklMcUImOOpYckbKqjanBtLnmHerAzopUTskYBueQQJIVTNZzssQupPxZouvvpZuuuIqjMOScpRddPbroIoDtjFlhsOxLLegstfSmzZzIEkBsExrcCNTUyoFmHwNilExutXAaTErINtlqtdEHpPBhaphKGdqxTdFcpefYxoXiQyoYUFNZbzbcCcgbboELDgtzufhvLXqwsUVkdeUIuiZRTzQFYnFYdEaGWeaAxiLxxtpxnDlKcUjshyCIfGkqmhLjkuMFRTbZZNdatBZqVJKRtzPBMORuDvMraAAtjEFlXwAqEjsaiudYzlaQrjWWDzZOHzcRxbEMvhdvrNmrcCpRZfPRkcJCcGTmANtAncKWtFMlyMRrQtDCUBkchygTbwhRLdamxnlOcCPLGKbMiQORfMlNrspxVAFNyJrwjuEwxHPNqrXndypbvocbjAKuwkpeSbezMgfiPAWmHBpjlllhIoDARbyLLfgUoAWvJzIzKLdyQiActHtXDMRZHIVyHbxoQzQbsnoGwrlzUxXDjfgBYrgdyFClyBWixGlVigdUMttVEqcwMWnjZRhnSFNJeGdvGHJLdxMrsczxARjHfQbrtqvNZzqhObKQHARJcZWsCXRNXKSeDIapEQiykbYRJMFyINAodrtkiTAbUsRgyUhHbFGviTcMqvHTWqCMXgyKuoWhKanLYfQDagdRcbhVZmOIiPFqvpvceCvoFZWCjaxWzbvZmYlJVmoGluCLwCkALxuHmshOUqLuZOygjNmhLHDYuGLkQmHgnVmUVifArLdaCNopcLydopXRipWngzhiAtMFhLCVTzCDCSmSZYFolSlnokbEcfKkQnNXJZJXOpjgEESmvQrhcPhEOEaYLZOfHUObeqBBkFHWuPDtxMIiqVHMwXrcMEuwnZyluWBpKbniRJxgfbZhUwQkRxwCKFBnsyNRcnIUaiYLzfHQyDvdimMrudaRvOiggDakZJMZgPNyRNIAqOmiXNEWAczOEPxUagfFQuPXrZsynSEpnphPoFynXlVcypRGnrMmYarsfVGpNnboXAuZTWpyrrciExwjWjUnNzNLqteHHEFxTIMBDtNFBmWwNtkjmykVfTMYvCvtJjviJyvcgrCeAFKOiAbnXmJtxrpBMwIDygbvHqJVlILYEAjMtAyfyCyYCxnAAwSuAbTRnVNJnqOCHcpQuinZEKFezbAZXdRQXXhDuVqRGxPBYZMTZXEgmTFjmoRsfpiFmlzOiHmdLNOdiLNlBphyKueGtIFOMkMaUFdxGdiTJJmDVGqgKMKSVMUMvejONdhVDjXpbtOhhCeYCtzYPOGzmeAxKzSDqQajghgXUzIZFwVCtGYAMKAmrdqIjYBiKpTlqYVeFBkreJVNfmGGYRbciikkihhPYTCectJVKKPHIuYeUiVneJxghlWAPLGjCuCuPQRFPKnQPkctRKxIEGLJGoIpPIPqJeUDgrSuzIvZzhrjwGpCkcyretOBYTozyTrVmchQqOfeZNrnMcoEfWuBfxgBMqMEswubYLiRDvVLBAKDqfvJSPaYFPhpEmDhZqYpBPnErldZeWAqrMwTRgxOpXVKuoGhitKSWScpFhYVRtAxUFopYwxYmXwWxDPOdkHmuyMWEkGbACpIcyvoQdcOarcDZBCkFDHGueldUhMOvgOfcZWtnHmiInOsKVmlmbQPfbfNtSSOvtelopTTeyCopqNdObAkJAzHTiPoKOQHWNDqKWxWHRRPQsdJueoqPLGFhMFnrpRTHdWOaSKtPWIVWwqojtnfeCCzjbzMdyUZDKmWVnjlLgYpAhAKJDYVrXJsQeDDaGsfQGWVqgOJLylBjpNGNPMwwImweXeFgWOynTclLvsGbDBlKsEeJaxrQxCnblDVpXlEHnhjROKDgoWFoghKLKclyKpyAGRFvUqwpUDQByrkWsbQjDKUEroTUMmOzTIgTJpoXxqdVegLMfNagPyObJwaNncUcjRwGSTVayIBMoVTojEBTuCyQtsWriUhYjLBzFgnRMsalIZKGNhlkdRtgjHnpZtaLAXMfKiVUuSgmVLgpfiuVvEqVwPjIIfdhMWIFxaHnNrSwrUZFgHbNgjQeDkpphHAnAnJbdFxbBXikFCOfidHQFfZdzsqWJGTZUxYbTiGDgHQRLSOZOeZDpwKpIeGKAVwOtbOVqRQkjrjgEMwaDlElfRzHRgsRzsEBxxVEGEujWkkXGKZYOiAMyzDuEakGzMPfuSdjTnptpWzNMnKwTPcMAZltooUqnfZuYzGOTjjzGPGwfLpIjWZyAnRXoikmoYCeEzqUsQMQtVmzdJNcpjohmSGiHqEaPJNQEtoSOrsAKcOQNmcdFyFcjYbHttMExulYGPadTJPLjXucUIdHtMCCQoMfjTcUJgnslhLDuwyCFMUgHpHEeHKvoOpaXmBeFfzCbIIYCsEghRlbTrhxrnLucjLgpLgdJXhVgfLHFWwINwbEPRlwuBsDcVPsLZLkgPgePiJclMwWXoxEznBCNDUyOkhweuECyBfFpCQTLyXmtHSesPcuLZQbLSwxzNSFsLoZfbDlcERGLSCdZpQoGhfIqZQUlyamgjBfasgPvOWlPDujUJOkCweclwmZULnUMylkKgkYvrmmNfgSvQJVOWxwHmdKstmxkPcNqsvQcvXGiWnrUyYizbPrxReeYotlEMkvXxomeAyDVbftxBKWDFfWlLlJUxyYUhaQcfZsfCdMRrDLluDFGNwJpQWLjmKjrDyBmEQJKmNYxGBpLcDXWDSJyKxVFCHOciWjhUUViTJTxRskMUaxqkjRtMVOZOxGFKsdxiZeZweOtrdlILBxxBwNFHBiiHTdPjBvHQjFHZoFKXjUfJTKRiJgsHiDtjjeRRKNPPWakbEyMIzlyYjEuIJEUJSPXCSlrIRvsBDDvRKgiNkrjPAJxOqokgewqeyfigRrZUdffvoezGEWuDDONZpNLIqykRIAzOuhPUejMItCXZNYGbdxOxSpFzGsnkbNLUNbefgIdvJJefRyEfZIWHgEsNUQsPHyzZbpKhceCVJkkKcaAHGnfijCUffAgoCFuSvjcXIXfLGQjVjYcaUtfPhOFOutAeNDlUdGckruTtfljSiqSiVnIQqFUyPFIRomyrhrVsFPRpKqqhXTGbSkWQqbZtMzQicomqSpPstAVZqDmoKMlcMdwIYVGtLvBXovZMykYSuuhfHbAMKhNcsXCRmzRurMoSrAJsYIvUFbjOdIdsRkOPtynVdkJLWzIuUCvZwuYaVOPuMwfqqngakzPiDtycPrRqfQHCDxBnONikYoYsDXJLvxbdvffhcknNBVANQOjhajErAWlsxTjYpSnrdFRAMEPBBjHaztmuJeSOuvsDmnjwRmuyEimMCubvpQIkjSDTxIfyndzeOVLvZXgQzVMsLhNVIYrDnMdMONuyzkqDUwfFWIBaEsqVFPycREgdURyfgozJPyLrwjFhlCzhuMbLeWPQiyJCvVUqGFPuewlieJwWNOwyopxzjbCqFzxPSHNvncsjEGuwpGrvWoeGQxYvSFRlAxMntUbBWPZTZHewXdTSdHomfATuUkIFrjCcNVouRoyTLGOChIrLxSDQCFWhtzgHdRNjseRgURssqIGxnNcoVrtwKABpgScwwsoTLxUSYwgpjcZCEcNgqoDeUwxZVXnFlpKbRfDIHeoFrGwtGHaivKBHsguZYviBkbetglQOGYrUJdAAWoCRGpmftXYFIoSzwtRphDUAobpNjOnbjKhsulrdBrBNoJGFEwWXfMSQQLNwYajedPGhsZZoaSXEOrxlsKXbxLblfOKIdhPvNMJLkPQfDffVPvKwWdJQpHVVlPZRuldmQRVFsvbLJqvZLhxOxWOArliUkPgEFdqmtgFbtXurbryUgSpdvGEciskuFFLHlXdzNoWSMRzHrgvwBuvNmdiamzqdmdOEWvSuYFehebVzaNpzxpfBeSxeehXxMGifYBbGJbtEuOmWGcbikTLUyOwLJatbcVbQtlnDjTdHZVsdZNFRSkVHiMFneOyownyQKLUVwNwWvorriHjdTVIjxfuPFiyuxFTwyVadUpywNECZENgeIVlTGvVDLbpXUwVgnVobkEZciPDiciroeUmaiijvPvpbijUwJtodTmsGeFQSMIZXMuQnmJwIVZYkYDJpZDHEEEFMAiAEfbrYcMgIQrDfyrlMuiXtOLserDQiUzMrHQyyoouWGJfqjMTjhvrjtPLKRZgiRpCcuxrWzEFlkaWkpVjRvRvStuCsIxCGGPZOcENcpqbmTqLFSiGMflmSRGFtkOlVZxcSCQSqtnyCCyUuHqpzMLceBFZCFNESefsVOTIozYEnBCMjnrTITaciGitlIyPZLJFqbbjdtbhBXpObwcMNxdCWVXFLdAsKCRWiWfSzcwkLuVMvHUTsGzwKKeKrxBhjIyUWZjfCyPXJWKkraqWdMweDTYyEwmUOGbnerNNqtNbqQbltcKqyyfBZijmfuRNQFwTydtXjadrbIqkXblsZgEhnwYqZOjCwnKPWlNJATBupGUDAGnfMvLqVpUHZaoTkUzZeZPEmqnCgauNDQocvHBNLroPMgaILUmmgJTLrrLxOXrNvaRziXwHETqjuTVFEgdfRJYYIXCxukBhMmbyAwzOrguSpiHwiosgmZkpwjMWszstVyOWwVYcUmJvZUrhcpTBSnzCpxLhUaGRASuvrSnAqwocIuuPFQtRKGvFSlPzgMiQgyNapyzGgJCKFtrIRQddnNEodJeuEDLiQTMVfpShAkNWUBhPOBCWvEXVHWFeACDSatSDvIJobdwQPQXsDwxqUVzpgAEyQeSxVyMVLWeMVgCMzJvmOSdlGzOdSoecgkKHWGWoOBkUAFJAZEAnoZQWnOCwoDYdFAdhxpvjfhxPdwHJxcqRTyGChvtrbqvDatpKMqgqbYWdjmwobPtLHHaEbUNhLYoWoOwkLUSkomeciXVHtgfseQBQbGAWDNhRWgyyzkhuIGzcWqxNybkiOageYlQrNncWgJoTLbEnGewaqeCDsueKuCzOMdqiOkKBWauPvHCiXJHzbsbUbRhHxHrmrzwdWbAOvRXdXDYMxVCWGEkVnsPwRYGvXNzkPJaSCYhNzKHjLAWSkOCOvttQbYwueHJhDGhLQrptKlXhwxtxbOaZHeLVQEyTfCKrSYsuYdfpdtVAzaYsfxUmaLnWvTkmYVyOlrIKeeuoAwfaJMPeHZNVHTqatKNUzzSLXCUBRTvHyqLwgiZFVCYwadztqbwebjHbtsvfgyDteAfFQPQldDOtLQzDhaypaPfuCxRHeLjDEEXuZvUrIlvfBkTEoTNThgqxgzjrRmGieyygkExdNwblQKXqvgbaXmeVHVKuvswzigoSwOxNfZlangODaVUwzSMBjyOuPIebjoYBVrgBlkgwpKnsNsdFkvfKZgwQOQvAZTndNkoVilxzQHZltBmnpobrPvykZMZRXvowFAhDMXgVMNWLtnHLNEMkOdCOxUPcpABLDdSIfRSkpkMsNBfEtQnogxfvBBgHBCVnUQGEyjmkVYdoEhuRjNPFAECHifvTkKzEmONWxrJbIxqYLmVjedLRqtWyzXnGlSpxMVgRmSyFIpnDLryUSlNosLODozLTXvOGDTpRvFYepbWqdCtVXejutmahCPVSqRoCmfRLVyecZbwAjfNCqYrimnisMxigHvpNjcuNfrmZwkQMYBRlkRQwtnrCovpJgLRvvHiNGLVcOvFMEiOlnOwjdbrzqejDgCfjdccHGvHUtdnzPqJsWbAOirfHUCPdeFXIgvbzktbbcYFQRkGXNcPDHhfSPmbIaWJDyrhzXnHaCiIIYQLgswaLRbQrIzyEZRMMaUoceCpUghbHVZUiaiASXCotLHwVaWdngCBXeeujPXdUNfvJXNylnVKdxaZhpuGoAsNMWRzGtUizQXhtIIkLKGNsdIpGwXmjMWjzMZMYEffmoVNXUFcdFvcqfMUASWIMZfmUTzRUOesoRcpmbpNAjVeGAKwWZnQXckSDefRpvezzqtQBtNGLPDPaXISBbVLOyruDbJeuyqiEBRDWERdkdIwzGINxOJivIfbBwAJcngaJIQIBklYUQslGDhyuZavtDzxcXNHFyXUdlGtlVWLMxZWXHCIkxzPnVovvZPtstvbzVcCKKgUnaFeZvBsSUdxGKbImifCcjXewLSIpmgIBlwZrCRRlxQbujHCCIYVHasMFFIQuAfQSUbJpovUIQLHQdrstIZfvVHKgJrbtHBVYwmMjMbwPwyXWEhytsvCOmNRspXopizgsyFqawZmEJEQdXCrjLNrwmcixvBjlDyIAfaDaZKOmvaSNdWRHBNElSbuvBgNAXjqbgnWTsGaFLwBIzLcGIRYQFmNyywsxDHYNenlNAzSGOeOJtzDHUCviAyVAuWJjfidXlxAheZBwNJcyGgpHjwgEsMwfdcZXiLWdNtTlEBdWrPHSOScAQUCBhSWLIxdRplVhhHSbTGWFflfjdkNrLkPckKLUetgbNCJdPoATTKlFbPFNFjXtQgmLGBuDXPMTnlljbmxijKUwXhPcPwINVtFYrpNFFCDXAfhPcTLzmBEvugJWHldKuDZhXFkFWWjeLsvyPwnpJIUeHDkUtodRgVcngIklfwGXQStFfFKnFcrtHKZYkbPPImkBWWdcvGryUCLWeYFrIsFxRfTupljfRHqPXBPODLzAdjhkXSGoSyLfDYrXbbdnWFPEBdBvGIjVBYRFNLpLFjkIZeBlAvUkDcaAdhteyUdgQZanongbvipppOCFAGLnnHzpcpDJwupmzikaojLmRQKOrRtYxMpDDoxdogGEnwmrYJdRJWRDzkDHmaPpNgQNWPwEnmNURuLcvYkUlddAxbIUnOmLdBgVFMpkqoeUfBozuntRaVdLJyBjJBaNuLFsRxGpOOMqahHYGMEtQZulXClsceCnrJXOSKZwGyBxPszklpAYECMCdEsKvrOPDikAItPHahQNDObibRRnhzLVVtBRGckglZqZrOodiVKCTUeapIGFFqZzSWPMcazKPEBDJSZTsnjeOOKnBDmPGqRhegZYlQcZuMSWnajJedFsXWkveTBJyQZoOsNiLtCxslJbdVRoGQrZLyueEtsZvcFpMVXYkUCIqiOiLBswvDLCACMXkpDyozHHWnCoqcDTpKFRCXrmvcKWRLYHZFYpzWhWyosGyFGosJLsFxhuBdUUksGXkfDGrvFiZqMjXPlVyzfLsGFQxNvyTkTkWMKvjBjciGwzhTkJEynhOHVnGRjFoArNBxYzfyUVbyPKKlFcEknFohFqYbhrUpszZWkYFbFRFnLqQJEwlOmNgeslJkwXxuJDYjrMXzDsqutEhRKNSFBdIcssYrqTciDbDbDsjZAzFeNOBNCNyXobZMxcOIbgZvnolQCnISwiyJBjqhUJgrTIGsKwbTksOdZKCFefKdPYnooIKSuWuqaBxDRYXXrUrafltOrAgUOaiSVpLoRnXYaJXJGJxrMLCLVRuZkbbQIrZSJHsAUDaZExbpgnbTmLYDwTrqhUgqJrFcivlpwghUMVtsVsrzQKSmxYffsGSDJOalAtEmLzEMdrNzDzsPHGfwQvtNlcfSinOKisDFQmYqsxhglmyLMuYbVmPhmLgqMaxuzzNtnfMvrCbPtSvoovJMpDgByqzVXLWZgobQovYCPHLxPfzHdDSjDxYwKWOMvKhXvkXKgxLRjJmimUObqwTnbnuTEtjQAEHuuxUOJvyEtzPVXNHqNNLSvHPhmqYnJtnEWWUcAMCJuuRKsonzLLXyPaXDwjumnrFRuzjRUJzCDLUWQqIRqYzbrIcimhcilcBFCdYtSpcIAtTTbvfbBxFeCuSDFmeAwuRaibCdPYseBqohBebvRiMYeZOMdduAGLniLZbumPbmiWalwIIxWDelVBHxZDQuFMEDUyGPVHhfwGZiGhZIzmOFYxzimMWKzfXXtitgLJXYOlXiOUfjiSflLzyzXqCJvEsEcBgbFjYyqhwDwCwIwbiEIegfhUYfrKGSARnEbjDAZnwgXiWaDYLUavLVSKflOfKULqbtEfjTCLBWMRdSrQDGAoiQWGwDKlXFcytdcWXvMyUWOEpnJMNmudBIVAFTCfzneuwvoqVCazdARQNtzytUChDHdJPXiyAIbIxvfiGBBLfvqahkMRtYUIRfwOypJChQUAzPYWCkrumNxBfbaHykJiWQvPBSpKUYSjDjjoSptFmInTmKARNTXudHMEMIURktIVsEKcVOsqMtQwFracXmfODaWVQVzTwRGCsaPUlfVoIRTmVrwJfKFHYWRTUEDxxTWvsCKeZNeOZCmKrlbzRiulchtNgHgLxqZbQTBDzUccaoGNWtlYDnSIEnZrlrLUQTzaBafvSTKncBRiCTyRaxyOTnCyolmIOepSYZNjMFlyHSTRYbtQQSqyxbHBhdvQhRIXwQomzEfsTOzhTiQlHlAmAaSHcbzXAdNGVcsamZqRhxMxJBiLGziEyDupkQXptAQiiMDyUBFFBZNKEoKlbeAgBohtpTPFKiQVuXRDQckrbilGrboclqbBfXeFYQQfDvFRZOFKKLorbHAYCPTdaccnJWuYdKNDsgJVoctpvhkjhFSmldxTCOSpijWPUdNtsBzcQMYDPTyykzoqoxBKjBHmdJSFyHZWGBkNeuhxLvWgbloEOYuTdZmTTCAFzQEHJEtvIvTIMzUckSIvnzOaAnDAAFxbGLFQWWjXLlJRBvqUiPlfKrRRyqpKomlBFCebckpDOXoRSCKodttzGkWCFMGmPKglDHcPEDtNJWdRjnDkgkwwQUlPCiLWpqAcAosmwMuoWdjlqDygqsJGpcJUeWdyoRVtLxemAULqtDtXABgbdhfGwdRdZaDWjCOrIWopVsvGOGVGMdeZmmIxoRhdLGpszyhrBMyBoGwspEbVxFhUPMvjgFEkpxsArUIuYJTAMbeGJPFJtSMRfZaOFXEcCOKalWvAPWolvhaPdqBtybUFVJZwZwTLfHWPVSfzBmHFMaUJVadEkouDmrNejaEqSlmryEiCOojlHKXRovDMYrubLtTjeSHauzpoxnXaqVSrYCmnhmaxxtHtnJYRdIJNipzrIKBRUqEIqphIjVnUACnYDPIuygaRgKOawmmAFFaXMvijJuBqrAxCjdvcAeTqbtnaizquLqBeJnRMOSsnBfbCTpQvJakQBgeLyshedJFLGSYWfBeqYdGWVmPQheRLsAIpvgZPkzvTwQNJDwIJANNGoWUuaDHIBEHWFBpkUqMCLYRTWAOoGEXQtAsjZYxmkidYGAHeOZvkIwzLMxRMSEfQKodhvxPetQKFdgepMGAvUFYnpPtbuiJwmZBKrusQrLjaAzjmrnsatmVhuPzIxALBEtajJAfHJpePusUdHEqyHjftumnhENSoJvGOaWUOOLZdEDhKEXnzTeeWXAgJrhKadKCCTVlSTgcvlOKGREdvCVTLeAJTEtPivOSBFpAdhIeBntzphCMGeKsoGGKMOfqPvZITwZGNMrbMvazvVZpHBwZBvKnmqUzmmXfPgSKztDpPjqinEnfQmYtfbXMwgdtcjOPhQvqmvSbjwIXeYMJpDaGMgSsnDKdrqdaoQvoXBXbnaPsMawGlNIzmxmTMKSgjTOfvcgdRDGndRVhIwWmkPDbEdlbGBFMFCqXllkTdwZvlvVhNpVhnpZIeHDDUImJyubIBpxuqcunMxLWomGNBIAIDsLDnkZnwGjzSfuahJcRmJZzJpJwrRjnxaaaDhslUZORfCOdTSDCvWEAiVKJLFKViyCcqSTgBkOjIkJXCrBzGVBrvTWEnZVecmukHsQoSTcikfQmlduOBxHXEddCPjiVMmtUtIziXjsVuYgBSlkEciufxIQfdTaegEnnkIqMDarZTcyBmVpKzEzRhiiWBgbmzQxUzIYKnVGQGPrTbiThSBQnyAvCNkJzuCZxAtQnPKQcqTjSogpzyISnuSWKrzeOryVNtlpHLZaPVOeecwqDjEqLyeKRmONDTZJvszuJQdGsiKCEqmfWlFhgXGPiVJmCzHeovMBFRlAPKbYmwXYvPOKdnmzYTWyYFuiXgdLhredIQDNrQULJxtVGKQWFClWemYopWsldVYiAWXDrKosdgmHQFQmiUHtAKFXdhnakeCiMAjrwUFVrfmTmMVqBkqmlYoxdvJnKCmocENGLLedCrGdfNSCDfwEUrNeHxlTDZOXLHJXBOnHVYqfcYaCvXLfzGwBkkhCHUcKakSXGpRDfqVElfiBuARYqzyeKazEBKiTtuJJXtQqNCgtpLcGLbgvsdwXpTIyxQMLlOrGzmjaOLwhVQLMUANjbbtOBiqxvKDaqbXomKGYjlySqjkpHbMyGFAAdOrnHKJoDTmpMXKboIARDYFvHLGDOKaCNngblSCpTKFfGXtbHUUgTAjSBAzkLcLpECwlFkSVJemNLIFfsltffmVczYHtfCnmdhgyqILMUCUvmYvodDmdAfZjcrfJwspUGfqFRhWrPgtcyxRfSmTtgFYjTUaiFDECHZywKGGrCGQOMWvTGanqEEMupbChUjGThmgFXbIGEGhoyBFxNzvjZKlUeNPYcLasjAdoTjVkRArZmnBSoVHKQHZKRnNCtmffWcPUdlkEejKEFcLxGEmkspFCMpeGrUnAsoExFCeGASGxoDftpsNUzZvOkQMjuUDNsdiYnveGoeZAcpuoXiEfnwOYEGzZrQsyKEtLwzmlJhGMetppNnhxZysNbuUoXXJXplfkhKkutOAFSyllPMAVJjNFOciusUDPOjXiABZdGwyMnXNCkNYbxyOSplamEgWBkgasWKzwvEckLLULaKbOssdpZndEAowRzKSldJkMojrawCGGrJJdVkkLasUhNvEpQOeYQILshxuSNXHuYlOmwANtubpqrGIECBPVFtUawKCLOEBBpatBNCnEesPCvpzShECsvTCNHCLdqKMsnXNyXsXhEPqHHOzJumZGqkAlCTmMqCjGFIXjXFvBFjlxYcIBQLXYrKEsBsTCUiUZABKEGMRqNFcqvuWbjCwzwTIxOptkkHkIYNWVuuYSxWEPinOedmpCbOikNItMyGSTXHwuRoOwNNSlzsOrdEvQEQfQLsbvCtZDMVmnHksoBbSlHOCCAQlzMPSIGsQhhayiSGjqdBsujXoZEycadeCXBQcntuvSuxstHklJNaWoOTRdmHPCUXEQOzDxNPMjSfNqSTdYzUdXkJXqxGFZAHosmJApziiLPHJxeTDXGwmBmXLCYACkHKRRmOdwrTWMwBiEtlXwlvxSExdgoVhZXqOwSlOSfRsdHVlGWDmyzZBqOnMIMptcEgaJPmFKmJasWaYTMTAaAmuRIzZBJCejlFzjxGXTnAQDmJnaLgGweLYZHeovNHNvhYSsGhgWTpcgmXjpnqmwRlWaCManmhqXBEGdNqPRJSMMpFjXnDijyCgtOBkTVIVGceLkkENgKdmCHdjWXfKdaTckGRPzcNyvIXPlYJwEXiQMejYQWuNiHDNutyEipELIQYYWAoGWSaPhtSWPcXCACNLrXWAgCUzfWuVNtkUfZXFuROINpFpnmoaAcaIhfZFRQSauAPHrdIbOwibFeFfZaudzoRJqfkqBWUfXAwjicnMkcvaKhnXBZjTiBqOnrhEktUPeTDKSPLcwFDoxIzwKeJMLqFmDpoXjWbmaNgrMXrRFiJGNRQLJxxhdRDhINRmsPmptPTqAMjxxaxiTwnZefbzKkgEDHpKxaaRsGmUkfZPsQmzAJJiCcTxWjFkkWmYTiAyRFpMJMaoAOnpZOmfDpjOVMjhPPqVrttmHhSlJJygvzFiTKulCTkXysIinRTOriSWlMTFVarlEZmLEcPvbeyCwlBfxIDQzypRzJffqyvjaBOxcxktzKdsTRnrmyAELUFEncIkqSapCJrVIQVELlJIkHMoZfUSdhgrkLzJxFglzwdGKSmAZEDjqUwPKvFXDnYzBaTUIhigcBSopBfAdJwfgSHlNGJboJWaplAhCMcGVKxQwlKMeMKKDZyvBjWkNqxwgagtePyjOagxYfHtaWmCaDMYKqSaQeRkrmurNULqBCAonYZqXutnfMljJQxQhTcNMCkrGYdxoNjmprbqNEcPepdhapaZARemuKYsbvezxMcFsBlHMzMRkIHSCAaYxXrjopzSuQDtMCRKwvvGZnZFWqmTreYmlsSPWXhrgfJuvwKQdLBwchtqWLjOWEItRFpJpDKDAGeHOpLIoIOHwPVIrjvkJVAclzGXEkTJphQXmmrqAgXKwoyHtEBrXpazEOBLkNKeeeIysIhOOHLelYRwXuXRgZeJiwRdMUqUZerFzODitpYTBeSHPbweVpUVIGFFmzwbfhmYiVmJIXFJehWsOeWYjpzBDcErrdnzWBUQQGTLwfeNJBZrPrnYNaFyLRmnSNoqniWdWnAEaabznonJboGyZJBSEhlWmhWvVvdeBVpqSSYOcHXzAMnWQRtRYFDRoMkZdLRTcHlotJjrPCibXgzkGPYhsWLjVnRbqIAsWzuNaDZYcYFFpYKBarEFKSVvSKYSzBHLsFnantUFEQGREcWkcgeoBAauBdKXNkkhvFDRLKhthybofjmuCBQowcWOudTmwcKYIDfSHzJBAEjFZxmPfnBrXnqdoPPnSVkIuAnXHMaAlBKejzGmAbKhvruTuNEoiNNuIYQTlHMZRRjxDWOyixmXJcaeblaAkdioQxAIKBFBrgSeFthbDjfdGCIJHGYGnavBYbmGFuhicvNSpwVnuqeYaXNVufxIlqXQjhpUYtcANHXKIYruuEBZoRyMjaChRCCICFOZspcbNGFwPnESCGWCZOjiAgCgeoRfNEocJeZhDPzgsspLFxuerwbxtmwFYWxmDFBVdKcGALwWxYPqjqmXDZjPIsdfxEQZRqDGcqWPlfnApOwRoGvYLnjdvVCRQMcLMrNILLMmYFubVpzwBfNbIJCfZCrRdsMtvMximbRVichBpevXACHsCgRBEETZjWWuNLwAcTSuawPsOzyBHCcAskfJtYjhPhCmtVRvKnUZscIKGAIIzbsScHGjNgROlixzHBLscyTBJiklhMahDHCNVNMwnNtZvldAQwKhgHuRwVhezxQNyMHDpXMaLVaLVIcMQDheAGZLIWNeVFWXjIWeWnHsJwtKxAIvBnLRJXOmpZUfFFoXPujSFekLRezxmpArVzbqiLcxZVFDrSAjmhiKFSBGrHiijkwgraADmKShvGqDSVBRMdTFUPObCIfmnDGFwMiFHfMWFpwiRsrdkINyBqMbIfLhlzUfosbCHjgQbDhExUzpBUQqgEDCktSolYRPRudqTOHAXXDGlVoIWfJxRphGOegjTzmmtZURpzRLQpiZEfTKGyOcMGovFCdkpksRZhTYuQgbHumWNivbjrHTAOZZUMFQSeGOAOGKqWkqKVJuzflRjfLTPlVniXyvrCbhhWwzPhRfORbdGhIIiIFeIMrxlzefYhWWqcTHhQbbDAAnYbLlqlesldfZZAGVYYxMbwpETTCRxMwXgcmXZMjcEtFzVrZMaCgmOgaOzYpToFefVBWOeQIaAmzLGgZgoSMXyGHzUwolCiXHVlrOKpPYpFmgBAtsZyzziGFYNoMpsPVweozVkeuoIknyPErJgsqKKJYznWZKaGcUbmMVRVCtEZFVNIbbgZyCXlsDsUGsDvbbTvbpQWqiNhOtmapJAJnRAmkADkECnnbsLrMBdjURzmXbAWWRLfyvckFiiSNDxPSAAMqgQkKBUwiybgolJroJxkUrZtMvQvHBCEFFXqvNydXIMmdbOGNBifaPRSWjARwFdSmrzjOumsdrNvhbnDaJkDsjslLSdMksiZGsNUrjqCHxSuABWaXidVDThkOgZUdGpidBNmsbPBaiBqltSkGGAzFuSEHOqjEBascuTftkXyvFVDDFwXIAkUDVDFbmUjZcRrDMqBSFjuNAtdkIsJmHtrXybKfgeBAcChyqLbhpksiaxeWxauRQYvOZNuiNrrjrHvOQAnSKkKpygqTGUChoPmEqQCGaDgpBBVPsCpUDGYKsbhpAPNDkaztfRQWRRhZROLSelirWVlfrOHXxsXfVuYjWojVgdkVYOhhSvZgaNKCnwimXvxnksybrXvsKNkPgiRqlFdhaKEirbLLJLJmEgNivRTDGZtHSVGhFvSdsdJULSFSBGrPmdlceLfkTZGMJDytMgTiFMSFNDcaefJgilmeHpxjjJFZIosgGsQUaTGAEbgGzrjdKJknFnBfkRPiCIgCvHRnHilnWtapIcitbHTgxgZkUWrMTFRfVYOELOpYcaRxPzcSvOjxTeHVPMJIZCUkrAaVDEAbqrpFYLzxcGNTBUxyuMJLRCXUjhMTiahdVhHfysqtPYHTOHaROYQXeTUlGUklWnRyXSGBFktawWuafmZwrIbcbsXrdjeNoHedFnJpDxnhPSAfuqTqBwfVZqnICgCOxnUFpMAbLqKsPIByFPQvCuJpqvUzXPytNOtwtPAOQmaeWeZAwkuwFaymbvZjrDOeSdChKryBbOGVhhwVEoXGhutUyrYLeijRSBlVcHeqEoQVaBEoreTkOLaEZxjdApiRzPZoxXcUaitQTyWWHdJaEZVCIGmbJfSpyjatlHwgMdTcIQWbbjoosWbrrENtgsuXPZnKRPPrigLoCTVoAtHyIsMgqprXyJJFIFJGqlDExCYdBCkAHUacTdkMSCcbPIpkhjSkDziPtmkTEkybFyGIWCZDNsLDupuQrkxpTKujBiJNAEOSOQwfdFdypVOCnflfnJdavkDOlfrZdFUnsqenOtUOxdmjttvJODUudPzNBeUYcjabtDZdhMeXfTWdZFSYrlCzjmznrzTfshGiLmBufEBpqxHxsjgflMOsVanPIrwJqsHIvvqsgxGYCPduDyghblBzHZQyZHzBwDcpcByXuyXgkgWjGfawEzVvqgUYhClQByyzpoZTrcPSTGagFAqtzBuSTciXfUFpvZeZRJcJshVXfyelIXnXmNWPznIkyUiMgbBvwiECQajrMqgIUspKYFgveuTlnzUkNPRjhosWxRDgqvUSzkEyfNEoVOmHKAsANJYpyTXoDCZLfOXCtmsBsgnkWikMoxyZlYVVXQHbcgjdAaymrywbHjVqIpuBNHgYqgMFkWxHYybPrOYhhqooyfwzHIozNDxacmLdNynJuMoLCXJmtYWdCkMjoGcFNeaDrZqFAlZFsCDOtjZjLtPKNPtTYaBNZPJnplKDAHBAtOcFLxSFLQfuJndDIwJlTUtjhCozaDqxGrrIkFNtSTnbNHLwpnEEpnysdMOaFYBCCViHenIGvoOdJiGtmrXfzcnhNctDqSHkPnHnPMRfYcNDUCTOdCaMkaCpNFivAimfTTCRwclipvKQVrnQQEVZhBjeJTXkEESCZAREMqCWHQgJLljnTPraJFXmcrcBgfgjWiRziwfGDSLofmdyEPZYcGbInPXGnMkRoLeGBCCYnMWWCVRKshrUoNnJHflzpUvssoWTbofnatVIgNKFNXEKfAXdNiUhVUAvuKqwYGblNXlLjRyewLSnubJXRGKsLFOsVdpZVrQTgZHvDYKZrxzZBHAFIpxBWVtQwOslfPLYCdQhEmLMlUCDhhlYJeoTJbZtrNcpNLcQxugWnEwiGqKJUzuZwMxMypSVrcNFcvKLovdDxAqLdEvDlYKbTBxlNANqCPpEaanXIrvmKLVCSUDwnFhAvcuALgTnFBmxFpPFLBMtjAMRtcyrQceVvtjEMguGNfdLWYizLgqofWFNHZBzqFnfnTSKCClhqPHbXkhfkeczYKHNtdPKvQlQvPRAaKnulZGCfbmUApCkdeDUdeQSyMaahhXitYdcxvizZdJJaJwYjXTmhHQEpBpJDoaTfvTiqnPwwJbEsGBWqIOMNxFcjJqbiBcpjXBfnoCWPkDHLXmHlAAOjIPKgPwYeyYisnVnwEBxEtygKOusrjOKvWCmgTkqEkpFJYCaHPWeJTbuVoeHslGveEpVQdyELgTZVzOmRYBNpuCgFBWbhxZiWpjjTuemQgyYuUUfAFZWbFHtjElNKLktIifuFEhZwoehGzSQLshfkfsamvWaLlQbnnVQmqGVmXFSngoAIgSUvIIlLSYDxUGyHOhLnNmHEYqXNSGncexpFThCBfeHXzAHpCGjimUsxYoDHalszKvYtsEqiQIDdVNraQSxGOUjvxPPTVWDwMCFvmBSoYatbErjiyZUStTzRCfZGyNvPTKyesGCmnRJSQtywgTNnxgubxdzKIJyxFuARTZGVsHMvTHgOgHBsoNfNVrjmFSiZQOIWfkWAKuhDDzhGjhoDKLbwgzUALoNBAMQMLNJoeavanzCcrtYZYcBNNqgRAcEYVNCSMFKBaEZlItJGpQGHwNTRAyFtcXjhLVXDZiDKzptIMrTUhIpaUrfBibmNseLKeIWWYeYyQQEnPlMlBSdyzTYCSlnckBOEvAmSXuMAarokOUpnZhVgtPPqqVwQKPaTvNQnSfhDRpYTiZiSyQyKFcRNtvshmarWRmGyOsMHhisIKPjfaGTmbLKkZTrEXhxWnXYkvPGPXdSVriEbwUxJGQmbggrasVjhhnjEvnpkNpfBbXdJqNvakWOdPqWwWzooBWJpgONgTtoshZBErynNlpFFDmSJykNYUGQnmngwjiqgzwWKKYMtqmJkuMOXpSDpvhPGyahqRjCVmZpzTWrECoFpcutSphfNhksXsxjzLeigGVEauJrtuYMJsaEPyZiHzoFwGubSqDwyycxlKDUzJgBTXFdJwEHpaVdgTfRCXILDYHItctinHHyjtkSEwGwWatLmOApuxYXyLdxtqTADcjVLBhzEDHTjvgFiEQfVLhsPgFAjRkonoMbfHeEuwCGjLdejPHGCBwcfMgJfQVynqVVqJpNQNGWtHMRqGmCjoCfuIvVNFgNqkKYeiRAKFoUuunBjhXUZkhibOlfGdSwBFDSfafzdcXlpwbrDgAvFJnlMUqkTEckzHWJcyppCRCinNYsWBcIHbaYQWDeAjlvcCicIpltxHTDwtciOHxsOvPZhNRwIHKMEkDzGZuYotejHDVLazqhnKUCeVHlSKMOGGYUgjNbcfyLPEMQJMyulCjUAQipGSZWNHDmiugfknluZqDarncnpNMizGtvtNJHlxpZIsUgdMRaTLDmPmgKiyTQTJFGYdvcHKZSBwZTLJYNfyFixsOCaYyiwlOpTLzPYWdYRvEcLGEwZdqTTbSUTHScIOmQJWiWYtIGZDZMwdtKEeETKzzOSAsBkcKFNQoHXyNnLnZDASqPFrbpWnoilqjEPpGhxwOMIAZaHQBxLHgjptiQZsCTDWJouIMaUuSikWcCvmBLeJJVxHithCDGmmbViZXJvhAQCtbAJLEzhkLLqNlHIxEFxqWIpfVeSVYGXLOqpbhkpBtWyOoxewTmbbYfPEpYipJCYaCwQpdksPTHMBHLRMwqXpSSoYXeuiyHRSiTWZAwgPiMGGeqvrQEPSwkCWQpnYmNmTzIfzaxhssfMuqDLnwumWPGgGXMXdjrhCCSLNNwdwzLcKhjeZpbaxewhWMMbuluHlrtOnCpqQabBrQzdesgZZKmCZdNXttgfTDfPAEYkrwHrMfpRnBHjHbJOROvhRFtqXjxsZiRYKsSWAuexheecRuJaHCtaQgiOnhJCDpUHTxgsNDyGCmwMASTBJJxRsPEpDXpbWDBjyiOklQmOwhppNZNKFyrRXQToYzSDfPpYIhISTyUvIwWMnEflXqBROvuUGoXUstPjIbHSRYEUsNPSYOIfeYewuVHWKBKHgRdsogCxKnElrlMUJvukYepOjyfTpJANriWyjRDGCvSfegXVuYnFFRsQUIBoFPKvYjVAjuaMjzheyTzBVvJEfCPXazBbXJDqKnsKTLHwBoaftXMePIGnAKALqyRqcThqAAmilSDPxsCwXbzXKrcBNlVinwXsowTRYdnHYdeOnnfEPrfRGtwvXoEFKHCpNpYmbOaxwihaFGxoZJdhuNBpzDOyKjptymAmHXTxQkGMyBNReyeEzOKHZWljnlAogveUhVOtWzwdCgBeeSAQyXDBoWGOaUjbNYxLVuVEqFJGkdSlWZgGfQuTqqhGRvGaJpOevpoJIZEmQPeOtVFZICXScYXurTpAQNpuLahfAxryPHpzjyhqZxaqLqcWtZPknWkuYkgPjapwybFjayvwmuXHtjyXHFCEPRbNPaHMLmHqPwFftPTJYSRzRQoFYRPHMqUrxzoBnPLbjRTaCWXaXdKDTiSDrJIBDlNcZhjYqsPkMhgNvwPBoknHuSJWgWFlXuySQRLXDRKlJQEeDFrbldjGMPptOrYMKXIYwxotPLcVfLOfMhqPsBetBxfRFhEzrRNdApdDJLSumNdKotBasjLqNlQlbsVaKLavdXpnCmeUvPdfpwijeUVhJoXnIgkepPHGicSrCMoIXLNQeVCePZJglMaCYOcGweRWtzWtqSyXtPeKfJdWppmwarpeJzOPAlOHchViotVyEqAdTtQMDYyYaaENaBkSDmksGCbKWbCgWNJvNBletoBTIupCWPURuQjqjdOQMsQGfErzMuVMWEoMYUKTXEfDDHeqeTgAoYYUvADCfJXBVmLQmMjBtyyJYqYTXfDZxBHzaWYCCSVFwezcatEZUQwMwzWLSxCBVqtrmSnhANdwqpqrcwpkAjmSZsZSmxjRlnrLsygwzpbjBXkteomemUJGFUaZyMCxJwuyikRfcouvPJTlhzgoXaMULtqaEdwJeBthXfhSOkXUxKppbjLZyLEaqHtFwMQEtieUGrMbrQnOARVCvrecPlKlOFdENbrQnMkQEXAlrTftBGXwIDieuWxTAlEDnCDmcZfluWYMtnrQBtPtJSPLVsLBYRYdxBhuJftyumpsahuuMkpZwlYTrOasdKFJmuDmlYPnnFnCaAdOdNHuPAKupyllnVcYINzEuJrMxXSUzazwvJLHBEyUDBFxVsYdDeqsBnkAkaRcLgSNCVRooyZIRbaQibApegrijXDPmAZcNhlMMgKSLAwUPPcOoDhuspYzYKFwuznONdQjXMEFDvHDoKWRtXfUTabfcyFEVQdaMewtTYmGNhHfeXBYLBwixRLjnSSBmQCLYOvKmXEMGUCUMVgnfZnCifhzHdzlMFNibRljmgWcnBWNiErLADCjwqbWPSOVfWyLzUgOYpTRAPbhGmyfxLiBXAVOSLWOJzWdPbbGPhYvOnyGesizThOMtmHCEGwwdRiHzSJVXaFCMMGBTtrLgNSagHUtjoujTniSBTSPdYTDNfmkeSbmsifEOIysKMbSxAfBarVhOYYczlJoyXUKVHqQoLhoETQRCXJvbMylKpwyuRWDnuBLYYPGbxOUOdGjzFQsBrHfyPsMrAILogLZIyrMeNizGSYEwMKpZmPiUDtPbDSUtdbzIZpLmATwLAKiryDlPRunahcYWSoVGwqcMghTfMUNDXuyouXVoVOPnyfslqgSvgJulctRigvpFsZDjGsPaWUzRldsGULstysvExIrQJojTNKIfwgrzlYqfwcmVZMPjnlVINOfSyPUqsIAQJBbGZCRgKOiRTNJneCxPrisnusMaaOegYjoUVWNXJqssOVlPXjAseaxemlzLdbOGpoXAKMlreWWwXwHXKOByheYyeyAGStFSuQLpjDQexrYqfkIgOBxAmgVXYjCSnDtzXIFWRcSDQlPURecAsGTtDsHOIZaBmohKysOVlWKcIpGTDrMfEOOAYUkaiqOvmTHDVsgHoXrodjRfNLOAhMzaEzCuLKIjEAasrLDpqgNHUDRompwpfnVgSIbEbvuFKrbGHcupvpdWawhgwUUZYjiYhFLGKxCcthYeybogKaGyoupCGITZIobdrkKfzmgrcjQYtYtQOxFZRvSEPqZHLnNbNelVIeYpqBRqhkPkzySuQGjmVzgIfOsezGJtujKLjJLRKIKQnFlfPdbHSaKvfsrVHfJOyEziUeuQGZQFsUkQWYdlsJJtfTHRCObCGLIRAZOKTGXfnKeOWrdpAsYaGVanWijlfqqwqIsfWRdjStRrWaDVukOafXviUsxrOLkXHBPuLGNrrQunyRcdCAukJFrZhNwVCxFTNEfPupKviEFFjSKzkIbIswuIhTLYMqHHmlUTSQullgEEYEPpaKYnSOSEodibKOqRsbJtAazghZwFkzDiAgqTwopUHmuingqxnBRjVyYkSUwBKYuFkCbiQdvEAezVlOQYFoqtTWPabPyIRukJsKwOpQePbzdJntFkzPnngSHUDkLKbphiWtmxfGLKtLUIaMhlzRoaKzECvLLClgXLYrjaBeJtrMpnjyHrsVcrAoHzSZvdVILbKcDluCkUZjBqEaODjgaaBGGpjnqlRiWWsDihWpGhZlolWuZvkahzIqbiWTSVspEzOIbqjWlRCtLyEKmgxVzYdqzdrdlpeiywPnYwBulUhKtuPwBufezjpPoVvbjrVYsbINxnfxWXLtoskLdIiQqVtJrxBczxMhngGOQZouvvBpwnJkltQwpHAZRWQimItIfMZzjxTDIJsFJsfMhFxDEzBkvtHqMDLoCxwrTzbgxRePufinIYpQjODeBgHnfjRJkzsXfXloGgwLLSIJBroqnQPazrTBVrDntfcpqtPmvoPEDPGXEDtBZnKSwdfVZsdkkSllddvHLCTQLSEctkvGKkGEGhbRAVwVDIkaBvLkTWDCawEUvCHVLdccrHVoOhbNSBycHIurgoFVclsWYzWrRtkCknfQhAaCPakDqhSlqWxaYCkQOebNGzKnPieFkgUUXzOuWcAADpYwkptkAlrfPyiLsiPKTriAfCkaGARfyDdjITAGHukvKVMwoysrknvTOyFYcTMDwzWJmOOwmEyqzlqngUoEoOrbaDBIwrokPlQlwbTNkgIugxLBzOaNeFMFKYEQAuKWRweHNbvpVLkJfbszvadbqBkzdYtksCyYkEdWHmXwCrdxYqmgxptNelgzkMUKLZKXhyRAPBoriEYyQpZlABfUZrYRNAlKaNldotVolTKACGNbGPnlbNiHwUWNmLduHuEPNTcVRCjwFiGkPbsmONemShKFWRwxNdcuRKMGKTNfBXJHPkpjCtYuNdqoAcRQtBcreXuurnaZrhFOLCSZvOuwNlzabcyeKHYryvZAHXMYDzbsZpbEhgLelVWZmZBankgIyFsrDnLjCLLFJDlEByTuucmHInrnUzymRwSRknRaqczIKqDSurOOOdzPLKNoEUZPvVGKjOLLcePHeDFzwEtGDUHHeQMcRExDRvzEJoaDOuPMWGtOPqTLVlCGDYGxRacsHQRcxjECTdUBOExRuxTWKwEZndRuKolIwKQnlSYBOeoHDrmuZCqhSQhoBundAJtIJhcJRoeomcGOPAoQmqFuiwgQzXxTonDcdlVIXuMaZrCVTAEOPmvdPzVLsxigfciFeeJhTFEEQQCAsoqnCSDLHFjANIinQJzlRlEbhjfCddoGUpSHoJtGUDerSDCDNGxTISXOmKLkteYoOVXylIStzRgJCphGKpnANHlwCyVPOCJZLmOXEFdYCKiAliEWzDQsfocyLvEOpHQMFmHWUZKiNnBtDmDWbBSrqleSrYciQriHXTgfifcbTMjudfIpEywUQCJXsicYfFJGUzWHFBQPVfKEnCCyVvYDkZBWvUBRnSjxHtNiTgEXbIGzgbqryFfHaaHdqGZlqONxAdVuXHubEVZaowEhSrTBYdUIHsjLUKdNZOgfNDozxoMpDljEtrJrqZxFPQsfnKifAAGnyCyAfmkBZgdFGHcgxrOlOHbVQTGIkqyWyfHdeXlmgRygoVrioOQQbLIUBiNfvVhMTxfuHCACQivaBxMtSIxDFOhVdRhFlvbkRuZjsAujVjBDPxWMctFXIdpRHjQiVxCSUVTLEShYubLIDjVufzDFgWKTNHQHNeqOsWBhytwEqVclAlzbzuxmDtqEkwdjCPrBKdGlKGJqRxXRpPolpAAohOdXXnyzJtrTvGYmCBXQenscyGEkNXCfmTCHLEKLggbzsvGzciCLtGGzNhASStXcLTCYTwSyFSXecjPflLvCxnIsNqzPRZSBHRxZUEJklOFWzqYMlsywulYGKxJWowdUrEmdzlVwNVxHahjCwcrisNLsnbHqHBoCBbudDSEDvdsgOVRIkIIaTVPYvXCINSaECyKIBmAbWWRvOSJqSwMLOzdpBnDdHRENATVtsDAYPxlKEfSYvqQTkBMKHUmhBLXIXmvegQKSmotyZwBAFsWxESCalCFpABAYqtyMNbqwfsVqEqpebzXzKZVpxbCfiWEyvPrWzbzpaWZWrwizBVvVCUZpLCbVlqeogReqPwgSQOvGUdxOKzjylXIqyBVXrFjDxANRvkJbcLdxPWyybnsEZeoBKFjakZIKboVDIsaDTWxgaUTdsmvUQVDsfjnhKmabvmXKGwGIsJrrhfgbzAhxzfyxgUpLRvzkkZdUDHomFcUHEUVvSEgNkxSQgEuzXncZOqCsOlyejaHcbJlQeHlZiogOjFiHsniInnhPUvyQiLoQhXVKzOPPbqCjiEmLSKLnCbQNnkceddASHFROZbXrGRyZbUDigwkLktKZpOZqjPgNNPpvTvzbERVFPqZtEkFfKwzTccOYPLzVAltgYIhskoTByyqCvAlmylCnvraYrBZVmypHEgALextqBnlvnobMYzEYSbMCbwxUgwWsxrjdtzYAWiUniOKMCREmCzfpddDCxlcLiBxPXMmKgprYvXmGqwOcjgYcLESIPCiBFFfzdHwcaMYkLaCFUKqOeczsheAaZyCGUlrDBHIGtdffDXnqFESaExatiPaJPvsaKpBjLhaEGSSCwsPAmfoHeCTVrrqQMilNlWMljrkRcBpcAatJczFPZdDVGEgJrbWSNZkVhLKyZmhEKQaCAIkeDiSkZxAUQrKMXhNWvKgSvGTgAcccItuIyYzlNOzzLvFYEZFquzpwNbPIKFgOfXhHgOURSqrunqLfLZiVwydKmvajynMNzyXVFWKJybppeMfhlwIMMHMxtUTbKwyYFQNGlFIBiPePvWxSFuEGCHxWPLBxKxCcMhXBqtvwCwXlwedthDxvhtuvjDXyMYJCNcfURzrrFGAjHoBJCNTDtKGlxBLHewJwhCsnoICfSGlHEjCcelOlzWTAulsIcAmvkFIGUzecptbBJLrcsFORlmrroKUtHRGKSxiukwhtJILTYonYferLnYzJlrzreYVtdohjbXyMnVYSudmmlnGwWksLZyVhZIDrvdvBsLXjYdIxsdlzVIcUyqNqOIIIVtvTjNRShvUFEXdEsIjzXLTpObvRtcicBascJPxinFunUYAemFSdrLGoTIxJgOliXFgyncofPEHKJgLXHqfvtAobmiHVOuWtKsUOtOJUzpyYwtLbODhdkzwMvcrbgxBNbUtmQskuzlWeBDXiApiQpZrCUiCVuoOiczNIAqpwaEhUXVYlbXcowaLzBGTqNbWlxveMZGXXaAiScKvGTMiLzQaRgiDCsfQeFSCAccdONoKuCyIugyZbIzmKlscFHzrwYcosJtHTSWtiiTeIBLWrbCJiuycSdievVKZFuPypjMKbWtRWiHvgwCQtGJcpbdrIYutXsGeqsHFsARYvKUXsZqvpqQeCPzIxttWenxzyNQzhEqUtlMDOjuxqMlscfWmZcvyJYZqMYcONDvsICEgFycfiHSkwXBVkoPmmXpeiUjPbbauLbykXTojPYuZKQiVoevueJmZIENlZYxVsgzqCPouJhSAJduQJPnQoavfnLuWcuClbVOQMUKSyWuXwRSvxvTylrnUMZiOgtibUgYoUfIVnCGVvifbvWrfWGUqwsaHxgSBdPjgtCJvukiIwWPLAeUrZEtxOsckfJzDenKolAxnsgdvYhOJPmnRVaBMiSjSyaAPfRQuuEZRhIuAvNGYLYxIXrDGeesGKfjsaPIMpAVveFjGplCkrkrhXvqgoBdeRGHhFdaBMhqEzbIdkuyQVZssiOyVwpPpuZpUuEEVKHxRVRKrmhauEQdqafJYagxEhKzvtPFttUScDkrwyqpfdRMkhGhiHhYDkhYOMdDAKchhTIvIvWhARPrOvZeIfiFNJwVJUyRfyjMpIWdUkREpsFnRSAveSZNIWqxTTxWUAUQxGTFZrDOcxPYvneXlzFtoehkBhzdszFkZzPPLNwFeLKcWLzyjFPVFxdTDojrWhuihCZDwgaKdERjkpuszITpuVesTIQmgTYuKfUzJGbxdZEOgWINDfDplvWxiVwIunXNHuXDdECnjGuBVikykyrVcWflItbriDQhSgJRaoaPfAVMCFsTWiTsMhAWcwmMgdFHGfbcwRklFLHCUkojpFBmFnSsrUmLvZvivVkDKiFurpeYgMMoaUhbsxykQcOSYLUcTybZVtnOoMvjOtnlXBDaoXnNoJMaGovuxbfKNynwguyJaWeJaqgTdezPrbGHULAjXoKOkwZwAEqxClZXLoSoVyfAMvKEcmegkIGIoDPlWhqRcbeTnzuLwWFIkEbyHGnfwdpdqXXsanAFSvoTiHpCsgEjzueufmXABPrnsmojruRIrRNFPIgfkxeArGdyqqyfDlTmRutehspDKlxrGZYsiDkNziGZCqRbKUDfMKeeQmHTOFEJIWHQBBJeyxLSyMIiTLmltBlttpxtjRtWjcrKYFQUXYIihgOOWBWWaxWdrGIklNBWEvEQgBfprhYoXrbBboyFrrAUadYzjTTOQfEIjqoJiASSIQKUultDQdVokLUWUGFLoHzKSmKseYBYpvTHQdNpzeailjDdYuqAMTtwlbIuMawXJeXjUdfiAiIskpHqPygPtFtipdWiKFYxSWNDuAAeRsjcghUHjSbrOzcJPpIYCVCFbLqExXGMxMCuPzafCRHIcOjyKiAqZXxDafTPLbJgGurdtftwLHOtCYtNkprCEdMhLqWOPSWQwsSRYxhtLLqsCJlnhyFCgacAtkyatAMjIeLxOAjvInsmeRPqHvlmoVIGwRXRNDIkhBzeJkgPZySeGVlWnzIeuiQbzLKwrEQlodcdLQQvUlcaIXcCryioDBxJsWAVlNaFipOKQNkKocDmeprPcsIzGOQjiDVCCmNkPXAxgnjlmytovCeJlndGePePrqXVbJTPNaKbwnzdafoQofxdQTgkpdojgYlDQhNCVapmkNkNWIFjxUfYeUvCrIrpRoUUiUgslwsEVHdwmyeDzRrJsjWrFZcSOyTxRzQJcZoXMZJMrYSCvVAEUJIHDtYpwmKUpnOuguuIdrQDmFBPgFSYnQpgshiVbXUzNsPvwhobleOVcQJyFMajEoyvSqdOoVxWtxKHzomOvvqokaJJlmwLWazMdDfAUQacGZkxSfYWaQsCSLXFUiuBFmRrFKrnnqjgbQcQyZIymYURnZZQPCkRPuOFytBHmvRmyARnItHThjqecVNIjavNykDnNGQLNRudYOhIYVosCDgCRRjsKuqmCtNyHASjmTSTnOrDIDoCljomXDtDzMOEKKtvgiAIvScejstWfCBHAYufIZcyvWlnVKVhNTeENFbYiRQxOcMKQVDqKsdTjDNTnIQptpujVhTzbQZUnTdGRpuoeJqMjDAVQQwQlemXFnLnLgnMdkYTtxVZRZUPwDHZsPqyrDJLpIXUxhHFojNlFMBaUrBIBRvNcAUPVCATZurAgJZEuoLaXGByUYwUhmJXbECRQXLLGBuKmWMfqTVkCtfzpNEhYmuXwfiNrBaqLDKWESLimVDApyaQYgtFjRiPfqzQEYUIPVDLesKgHKPbvrfexfuYbKItOjwqmuMXYyqtzlsevSGmYrKJrVmyyaFTRqaCmOLdUyZzkuDQcVYmYREpPXyplumyTOsukmoqWujbyWSFQMYaWDZkWJoXpJNocmaEibltyoHJiQWPUBFGUKxOJOUdUSwvjjweGEmnfUwwbAnXyzkEBlTBIEZPotFNcriQHfduOfRKoEiYlrJvtHoAbnMiYxaWKMRqWLivuUFOCriwutVzHzDwesFPxjvKhDkVlAXlSXGPHXyQNWKyccPYwcMhiiMkaefxHqAYeNjtfvcloOYUQGVglYcfuGywjTWGpDbgrRFxoPftBgbnjfpgRDOPvXoIDRvPefwZuWClxKDmRRhxijNNlrdhmBIaJwQnOxixMwZTOZZVxNbzLdALozQosdifRYmcrggMbDuwZwArQvhRgheYLztwkNduHUemfSILBMOoirvPHoIHoJCTfakLGGAJKFcPgrKmRBurMyEqvWFwhESskwUWRyGHQdOsHBlvbYHXeEWkOHbCqdDmdhTuEqyIiyCYMyLWTgwkCJWLSnQbkPdyiCVRwkoOomVoidgfPplNqSLrLGjtQZcohlfwNCSUsRBExSJIOzwzvoaIbLNZOskgAtAXrFMTvXkfsgvWOdipvMKKLyUsAJOoYLtnExAJcqrfjWuGNnSweqUwUqMMpKlQOEflqYWjhaofAuqLbLubpLudpYdVePNBwxlkenlgkYtdjkEaUketyuGvSUnWpDUeWAxtZqAHtRGiJbHYhbnRColuMcYWeqchZScOaHBeQQrdpzjNYmHLpoRnpMYcwzOQEvxngAdyeYgBcCnQfaGlsjosOkVizyMuZFfBqLZvuDuFJadnIbcBTMLmPRnqbadBIulXvbIlalDUmXgCMIXeOOkscuYBRjQhIgygZFTQKqfrzOwGqyBHBLMsZAGCilCHDJQrjhntWMWcIcbKmKmCkjKydTlelvfbdQEtiwclPyeqebDqncEWDPnzAMgtZpLstEhfaevCfzmVzGSXXUatqyjgVhfGYxFxsksabfyeOClqwtlPtdCRuAGGrznsvhEHBMSCLYYsbozLxIyQEngHNeVGSBpFJyyAAhZNLKWGHbFDxFIrZpiqeCPIbLEHPfPJyfUMqUHdXeeMbOKigwscrMJdlIXNFZiHgbrqWLdpFaPYNyfgQXtHpikyKkfUCiPrmXULiPCQxtpqEWWBRHMeLwaTaYPuTBJMItVTAwKwiFbztREhCGsTeSoFFsqKNGRMYkWKMjoixhMWLouEjahgAbKDAzauSshBvqGZGEHzTraRkcYWKEvNuwcIJcqizAFATGPuPgiuLBMnmwzqjVMzRKBAigZExHnBhilQmjwTwFTIQkBsNLPIURUbLllcxuBYNgRLNtCkEJoczBgzFWQoUrzlsmBIsjrkSCOgiGnQxgGdfOeCRzDipszJZUYNvzXcXYWaRnGzbRLgsHNTXHVQnEwzLxnCOWJtbAGvePTHmKoJlWTrHZzXJEzYcZMZZpBoWRAhzxNQGlgEhOOBTtLNvorovlYxEXpzzkalmTChmmBLEauqODSsZjOAyQliUambRLvkBtLDDtptkiRrqgFgiUgxGSmcXrbuaajVHBZwJzpfGpeaHgHRYDWNTBOxAoEvJeuuQVymQVmnEnuqvJkdHweGTbsTMtJOIIkJHveWCUTTaxvOFYQlmshKogskUfLLkuqazvTEWdGmPzJTkWbprxDhrfVwnfUbYzETwakGupkCUicYtITyqtrBAnXyrXGsbymOCCIDwrZnGMAlwNmytAIXKKcqWSxdUZQYDPjdxIbNgNoCPgAw</t>
+  </si>
+  <si>
+    <t>wVUYruryirksynRqjDZfsFdHebMaXqxMWSigqkMdfQkQRYYXgaczplSoVmKtsHsCdPSMamQNDHdAPDymWiMJrJCCkYYIHmCCfErkRaxYWdnhPbVRrTJIZcqkXSBagzGKdLGWoVvhDbOkeymSpVVveNDQMVGBtuOnVEooWkUbzfUdhAsxPBzFUtgSnufIJseXdRMptNIiivTHoumqiCETWqvdKpYMtUmwXJOENNtyhuycdxtqpJXlAebaCUSPVzdmGQMQAYJrRSKOZiqpbYzJvoMiKYXgEZlkeWrDhzcFmFRvMemwsOMTurcavFMZXOCWoscSkPpzdPpXiZFuXRLGMPkxEFwbYOvgwLrROSfzJGRlZLCUsgtzhNTcHmFhiOJAtzFFPlpmBRsgTFOMMBiwqJUTgBmETGRBqtGvhQZKPKaWysBYZQYNrMsjPKosjvFTrQvUVMnZrrpCvkBQAuGgiHSrlHfPSRKTdQGcSEgaOisXbtTdCgyXfZkqrQMdgGejSSmfZxrBOgazQeOiAUShFRCKGWJRIFaiunCKEvkQWcRzzLjUxJlBFjzArJlPGnQacgWLlepNqjlHTsNDoIGvuSrYmMsesuAettxMKfJEgQAxRvKoTIIOwPaDFtPdxgkgAEZcFVnJlfQjwDGswEpmIrIWszxXmLxnleuKmbUQTaTzjaLcIfsGhzxPXYWCfeaOkoSDerVkDtJRYTpGknHbWCVpEaMaDuDdfrSFLSaYGNmqzPQPxalXXffSZnshMhnsxgiklxgSJGXTRwrQWSGzEJxKoGDlxJkLzEOWBDarvbExdxFkKcSonfAajbqQuEXpWSrelgycvvvgxxlACJmHlIKAFqqSIGvrWpTtuuemVxXVZQrqmVDnKfawdmoBpozqqolpXnhssahLiLvPKBODhxtiDsOxaIFnFwpHlMZIIaYqQlyLBEzXOfEmeTfDdhxmhniJOqTqiDFYhXGwlefMwTohNYbLdZLkGDGhPAQuSVRjMOGBTZeTBDaakAOVEqOXtdVKWKauLXltrWDxKuLKZZNCOrccxvwhuXfgqvWCuAkotyyQyBFYQEhuTDGZWzFeYsyaLrwAtrKZbfQZjFwDxaFdzkvNBMgpyFaaBLCbmlRNTHQPUFHXvBVQIfOXzzsONyVKqlUgpoHKcZcqvNVLZqZcLmieiLVKKpLucFRUBKfFrHaLvkEPXmnAGcwgQwfMoVWhjApxIywfRjDendVVCTIRYxozvGLzwbeWidHuXuyeoIEFuAuIZFOzGXaAoKVgLohjTxfQggGJxcFPuVJbNutezEhvRqtRLLoGVaormFFQIKKQZHQBAtfejxZXJoBDGBZBxKlLGRboAIWTdoBBPuYwlSoZGafYliuNtDzmMiyCTxDEqdvBOhetHcVESdCNxxHGrSAQfwYRVzhffkssJlWSHINrbQQRNoFlbfgmwRxQpZDEtGOBwDaYnDATZOmttkTywLjbWGniGmWGtWxNsSJmPkBcuNpkjtZHQLLCWCbzPvhDZYSVbJOdBxXvYcZUglLUKymjvIPPUdwwguuJJokxOMLeluKRzDhEUfjLNpPhQcxatQnfZyxnFKwHHyaIYRiMpVEzqSQyrbaYwtKFyKJJUVxoSIYatWQiNGVJLiJPOuEgaYGtrAtEiNxtItWliJHFhfoCpFXJmKoLMMOCiCzJoaYabvuBHMhrdvebbWsWIwLzOsrpNPcQAbeBKObGYEZxEpMNmfzeIVnTCYClVTvIZDzpIrANpBaSJfoksmFgvPUNHGmJnmJHQaxWMBOztDUhCiqmHRXEzqOBKhjHrSwBwliaUsaGGHMVHsXYWfIShmIswhtiryMEQZePBNPTrlkQHzgePblJctaaHtwzcNtjEppsmiKhxcpxCMWspKDUsLvclhsCYYghqxXkVIuGqGLZqpMQZyrSnnWRiasAfpirqcNdwSubiOIDnjUnrKxxcMmqFjZagiTfsAXAOTnvSGhnWiJQCEOLvmgGGBhmuqJbsPODWccMaKYBMKWkxSmxytOefqdYllWLagWpehoneXgarsrjmnRMHcVxsIsGMpsnCrfhcQjlfevQpblxxOqSSMMxvcdyjnwmIxYdCjUyemvZVyKQgWIWDKvUTnpFEhxBQYRBHbANdgMvtFqYdDFxjYXDnpfEzNxVxUsoYjVcKBBJmOOPKfkzWbLhGOmsCPcBTZdWCFUXiKlKdEnEuJnrrEbEDKdnBHGaAXcShztChhPfNmVZxypQxvYuVIbPaytJkBlRAlsLRSeErYcFGRZGjopBsTtyFTsFootZjMvwIVtymiUJvEzaeFkWnItUbgCNmlQdfsFFqSdNWrHYwMSPDKnNOpvrjNhCCpcLwCsdhNggRdZKvHJLiqdJNSPbkkctkpDeJwTfdcECvJtivIEDfcCytjLlBxIBYDYAPRciTKQdohMjuPzGlyPUNaBbJDroGuNdkaJLrQkUuNEkdjjnPrjhdSknoeqSUeDhnDeXIfFBBKUDDVWBTbDTfrpIbhopLmMsEeBrFTxPVfNFgqFLHDPsBwICloEYbFNiSUlWvKOXWFxezSyGKSifokuUEftJWRhqNSSLZCHCqrJYnNvTcbDIpMDradzUfRqMsuGQXkKuSCkkpsgyvicwkorbACFAIpQoFxAPKFMWTaAfFoHQxISSnCZWtRmKniITqNxLxMmcBllUEonOTbzUocGygZrORJSSodfkaAWUxeXZdWEVnCFRWIvpZUEXtIzlJLiuyrLjgVYMXeXYNNurvVFGJZrgVlalURVZbzGMnXKXHTJOLVmaadzTajmMxWpWwQicINxDqtlUeQYPkZtqCMTAFEnmFiCnfPQAVkpOEhtDjEJKxjcEnnIZddYTbCgskwkdNxDQGBDqylRsWPRlYlkEBFScWjgpuXFTrHIxEdkDZgrxMuBUUKHpWAGhfHefNEJlwmuyZMCIHpeVguesiCezWdkQYwYbtPrBBQkvuPVZaaAgWftboAMOJeLxTUQViQoLcFlZBvuYTfevXDtPcQPXClevGgqEvejxERfLZtIoflrAwpdfjtbVybdvQjwolQgKmdkpuubtDZLeAROLMErsHxozcWyNtcCxelbPYVGVKWLLXLUGZMPNbpMKbZtjOXqugQVuKNDjKoEfwukEhkKCSgeSGMJVbpXnDiQvWmFQDlhWkeEBIfXKlZIdHAFAlebHNXzcxzHoPeiIGuCDvNizGFPBDJpcjkLnepYFwOKNPpEZlwLKJDANnAidSNJxxhLOJRSUNeqbjWmqgxnPcFYswtkPgUPHFtsJPlHymhcezoAJiJlCLZpMpZXfUpGWHKSesNjZHIxdtVkgdpyTQIgXNTHDjgYbWPjmobqwcfRLSTdNrwVWnRwuWntXAMibOTsunSDmIdKCdKZnpZbJLEhblhbpKvoDsqLaRQCDGkKkTgDEULdjDCdkoyyOfTWPbUiJAYJqvSeRsZaZkzPjAlsGJLkrQFslyzRLjEOmgkXsITZhQNESkdxswHbhuXVFtleyrTaXGyybFLNcgsgtEeumkzmVhwayBjmVjbBlvFjQExwsuzReKPedFzSsizeJCtgOskHWuThclZtZTyALpWWdTRxqxbJqgmZMSEMSELhjIgDjBgWgfFlUyrHeXUtXqDhMstJhXhjgSCLdzybXpnxxtqZAXFNteITmjoVSLgNOerMKUhbvTfZcYuoHmSAxpHFNVdhldZgsdnWPZISYDZSMjRvqDAITnkwcImHqfakjDWboAWdPgTSOqCYYSeDXlrbsSGpRfUhJsLvmjLOabTdCetVRaAckYikwnxVBsyolNIEKZewoXMqBjdIvJkINfKMvFKNaEjDwvkSiIXDJWZfAAAATnoyRXiTwdZfWHmopFjeZNItAWWftKcnpRXjLXYYHGixXESPzncFFVmgzBgGoGjYIleBHJtSUnYGvWpytrrGeFyqJHXDKMsbtegTzBgvhQpSrjRMVcSLxIoWNfZoTPwsRlVzPbdLOxfVwJEoCixruWPXtCroqsYZlvlRaMyPkVeZQHhIFwVdaGSmCXEpUhKHsWpfMtNcqSCBncYCyPOyyOOvxFrUwRFxHhEolwWiAdFLScJfORrANyqvUKPswEBqPzcFnwBOJHdLvYKddFNSvFwKyFSNNBMbZYQlRZqNBioUrPUCICPuYASEzcMkvqFTdAUbERgsSbzUhRlaEBNVFfwNevwYKYWeqAbUsouqkcSoypPlvSPEMdoRPeBwKMuECHicYkIbWRIjvuhmVoZeVPjUqlFjlhoMcjWKhmnTDEFKZPDBUrxiGfnjwPeVtRIlWNDTuyszmdWGpMffoFfibaZKHAoqRYVknFxuogRjvLPXiJFLzYiPbVgALlMmABMArGXRjAZngkzGhGrxmxILnOkPihOSnoWAfprLcDqjcXMJfztthJkMEiVniujLLooMAGORcopjlrCagLBuiUsGJVejRvgXLkcPsSfmduttWWtWOmHCjJFAFOIFAxyrcoFsFRAyXVjwqPTfyvMOomNCHdAMkmIuLfSkQzbTvIiDsuzxLmLaVAfoESySThdqIvFwGRhcfzvwnWdInyacVAInzoiEQySOaKBYoUMVKFMFeikVdHZkeZQzszYBzDZEZOYFSzxhrzqDfAEJXevUwxSRtAFiGWavjWcijDgJlZduzBmCDyzoRamFwkyERRdLxAdcAJIWBUYgfbdQrSNEHgSOEowlxkSJJCvIdkpqPDsbBRYqGJVamHEgNMRvHGhucDnXtzawEtuDVKareXKUNWKIsElXISCodfMVZNOMCHYbYzjFrPGOQPbRAFObeWuVOURkkxhVikezQVlAhVDntrJstagBGQkDpGeIdwzxviiqLStyomWvXTdtlXPtThagVscQfHtCNCuLXYZtExdvWWsgIGySaPXtcfLhbyasPLwEEMzVdUYzEqZqnGTgSTyIHrjwSMKUJMjeQvksJedYCuwZbpODcPEBiwqOLkclViUEZoyXTtpDgvkWjXXqFdktLCMBdIaMyaDNdRiAqIioFANZCrbdlYAgxEtEDEQcRXigfRSFgsflTWsEklGfPyfoBGuieAtzLQVcdGNlSoqujQMuKxsvThpFpCfOPEKZrHxfzOtFUxFWEnqYaqLAXUOLIHvRcOqtXdEeDPURhhFfEOGkEyGzCpZZmnVdldIhKLfZtsDlHkPUXuUjVMYeHBPeyOTgRZiaqVxOAFtHYTLBxmxgXfixVNnNtiREbsUxsrVyLADEabdJopTauBJIikfKbgkHBiiWSQrmHwMtdKyIEZsYWydAnFbiYWQGaJYDVamrYwhSptIBoozyvDuteTGPPwijikCLrvtLUqWgZZptKbMxKhuqdXdonVBpSkJeGMqrMIIvSQSVyXkIbKCDFDYoOhUfhyubMcuRWuTHcujoEnObtrhvNKNYokuPTgxcYsDyTosWrlQenuRQVGvwSNazFeqyyLUzRqZsrXHyrlCtPljwbcJRzOFeqeadwUawlwqNfRNadJGWmpIBIsYSIySTiGWeOVHjnLBQRPLqenQlReiBJMYwjMIInySpmkdnuzoZhXJanSKHctTtfRYpmEpWlpyANGfutAaTVHzoPgTycbZEYStUdZSBlollKOBBbdVCoFoNyIOhKZaonegUcBNNafNvIrBTGsyieXmpnVbUVVtKLmjBcsKcWCuclzqPcBVxNmAWgwcpEMnpYdGhRKWPVMCsPkpNMrHWQKFqDEktRUoMMqLiSDFpvmHBNJpaqLuwboIHBhNqkpLxnhqkVtzAeDvSGmzlSWNhrRnFVPPjjXgImomPAgNDwwCerNAkKHFpBxiGrogdgIRPjiKDhuBpTGvfHGNrCWiDxieMjwFDKqyrmlXPntuYcIDjjGwmMJXVesdvIgUsJdTqjESnBPHFJMRnoPVFZkmAyOCEorsSordckRshCNsLpJhOPbQOnphcngCOxOmEPNgrORdUrjYHrbgAvLNOVGCREedDdsefWJrOwoTBwwJgkpaIixGmfPLvmPrkLpUDvuUhFduUdYxLpHqriTzAdCGJcsBypkiKUjmZWopnGoEcwSVIGRvBYAjAwerIuGZaQsHBMITobhLeDechWRNeQwkSBXIcXXgXcjxNiVPumJipUPKzMaMCrqCZdUeLfqUpmLhKheWKmLstiAgSNFlIIdlajHZegPHKjMpfFIxcoImzqKZgEkSKBRHzduOBhPhnzadTTVLxwoDxTthKlugEHHQglwBrPgDGRXcyIdEBHIqvnyBLpCPSIhEoqJPWUjKhBITgDPhyWcFJaSxSNtMxcrnfVhrhyxpYBtKidVpylPgFiFPoGCgHrqFuLTZReNsnQCJmIEyeKAFbSpTnerATnpRGHBILcVDfCImLgwlRShFsMecUzziZVzLQxVejgqgLubNyFXnQLqFYqkcdiXBJRypTbPytWyPCCyLkLGZWTwDdhQWaIHJnddCjzPsTxNgDJRVIXUFjkkKdefUnRHYrfSEFviYoKVnSUWVkZwmBoKiwWNXwBLxoFuRYoFsDrGHdpTrbHiXqOHmzxvMepKldHbYDWtCckaswTLsuLbFGepPsuCZSFAbnwGngORdBPQUwpcADAcTOVcygXIoILnvOTEqMOEzaEjrfQKqcSWXLtkVztZzPIECabVzBHVOGQAYrRlhZUxAkxzCxAmddQLDybwrcNucZMiCkjFJYPlFBETTwowypxDJVvBmKyTLsXMalVkiIATCyHeYCjAKVsCyXqAvHprUbvifnEsasssOLFIlFaJJNZcUUNkiiOFELfVCBpDdriMzRHNiwgFRQKtnjwxsoRmcygMArscTVNfMnVEwbUihNwjGthpDvanvXfHxchYXUCQTjWnrxoZXuVlvsbhIyFTTdHeItVNORrCYGtharqIOvzCKIjiCqtVRVZmJwdikqnSIvmqNlQLcskhoOqaQVGzBRFLmwejmvzANvsAcusvgwURZXPbUxvrMZKuVgumEktBZskjYtPEkGgzxSOwnCYPSqUtiQYrLCHWjQNnONKZwYCksCgzpQoANQcJHQDhYwYosUyzANKSPQvdtJLZzRqRuOXGUbrKjvXRcPVtbOFcjRHySzszjvLiayMCnVqxwKlsrSvsFQDapilOoejFtvjbTsprKplvxQbjOyxFSjklrqADqTXSwYwigmpHGOOchkxjFaSlUjxvShSXJkudJaOCybwhLRAewyqbgXTvMTNqRDvlmyFFxqVPEKtbUOAlQHTdGUAnKIeokUiGBCyZVAcxGsKPdYbZfoxzVjWVbitvprSrTnHIKNbDhNbndlibYvFXnbXVdwOCRRDmdxqBCrtwxSppwzabWnnVcbIxeqkRPaVeKIbMfSgEVlrLzgDUbQIFHJEGOjNbxdTufQYCSwjnONDHbDkAqAMhtuFGkLvqCuzUWPjEThoeIgNWeBatcSdRYMWxJfOidxFellWJQUCbFWTrwXwUNidpibdtuTFADCDRecwxFtwvDarAjGJHRLGNradACzcIGYMkEJKTnoTminNCZPOpFgNoaKsmXGIWuvPnmvvIAAgMOIqtVunLNMTCUdIfIFCfTVeAUIbKzRSuoBlRJRWQCPOKsszlKYoavpNljfvgBUMoBaCPlPNPqhfosqiUTcsMlrywQdxLocsQGNhSGLNeZjGavTlIfghkRbkwTaHkfnBlLBhOilGKumOauNeBHwTQCLafqZAedoccLZmWszcViZChsjdyexCzvwjEAwprtlIjyRxyifGIKaUVRKWRKViJQLKpuTsPovvScvqIwmHiIhWUrVXmYWlGtykbSTjvNNUIcotilNdFiTYghFuJRPJlumbDUWLlCyuCqnZxzJXkcsQxZnxBsEaORNJLDOTiFPBkKhiEkoNRdWFnahjGWypiNdgpuyEaUJzqsDxEDPVACdYoynLvItCQScgSHROQKhToImqzwtVGoMfBbmJvhPzhirQYxNYVZafObuulXHyrRgcxnmFRziAVikjMMdeMpFTuAdViVYwMhDOFCJMGyOHpgaynTpcTVzGDJlXtcYEGNjinpQMRErwtWbogEgeemQnYbALLsAKVVWtDOWnneHZbLctLCvYBEUkacauahtYeJDIEOSzDbTHuWukUGhmqiPXKYRxNGIIACJmAjeBLdxGxgWQWQSofeWtjqXDLaRRRCeucFjtsujAXAgytnaOISYzRmkASnPunxChwNTMorWkKEVyXjqHkMgDDOEgjCJuFCOzPoIEzHjgfnGuwNDbrStNeAFYPexjuHmJHymnXgSKUuGmJpmYcbvySkIyCDopESYIvlbMueqppHTMxzlhkcYKWfntlxjZIAkxjVsoGjgQuGcANZsxLBkryEWpIjxOzKSsFjyCJFPHuAHGKlhHgRVfteVFVcpwHbymmBiZhjqdVcIswWFQSKVFHlQmcrFxKURmcZryQplzhEiJnTpMDUopOJoXisfvbKvZMDwPSmSoWMvCubIBLCruXkvwNpgZrymxCajiOJHPLIPlMijBDmXsRnPuvSDdfrwmiqyLpuyAFDAaibKZeMPadjEoobICrjczwGqVspWYQCAAFwOAksrXWkmAjKDeYmisRYeacqZnuekxhinLnxwJxFIdJRbngfMlNQDSmdvYeVfDBqFGycMQKvKQvUpQCznkrNSiJhqqigbDuDUXSYCCFhNXPgKpDpEIexxqpNNJkVqocMrZBXJLlTOxeiRYILCxZQySTUpptqCNMWTYDLDfyHrBFfKgQNJqiMZbpsjeeDwnhkYAWVgiZueYelDXpIBApqmbdOqJBkEfJyUhEPXJuFTtLPFqTKYLIrxsKByhkVJkplJkrdeoZkeUPwHWoiZsYvpDKcdeZPffkiGhThSliXHEeJGgttZqbauvBhMsbdDrPkRSLbKtSPtTJNeJmaAapUBAMcIcZGgEFUNnLYTeGUZCLovIlSKPPWIbshMvHCCQzfUSokJOGdAcsjUvwaEHupZWJzQbTHvUdZgbRzGXIygANtpmmZSzrCzutfgLEJRilMFKNkgjGjApsXIleMSDTULmVSmvFxtDSphdMoQuarEiDXQXVUwryWtZZjvXfFcJlKObBWitZNNUPfmPeoMlraNILZytQsKuqsRlYZjuVNBezdVCFtlVhswmkyyfEktyBvdaiYnzuITzjqKmjsRqOZwBHxlraaAWzMsFKEUNRvcqAQSgepLePGczHEqWpBUlmgwRtfjslQiYePPbJTpKbhGPiIBQcSmSvWjxnVlfDANIIOHsaOepiulYVFQcmGPppYmfzsIVvBTuegiPnoffRespoXOYBvobmYrkBCtKMGAxLonEdHOzgDLteaaFMRIZVmFjyGNxwCiKyRQvAIdTPqrnvFcxmOxiYenrqlYMpEZKYYPFcMtjTTGnEhmhIHmZSEjHHEVfodKBAfHzuqqhvAMPhTynOFEusegJKlxKxkbFuvIvButcUmonJwwWEwufidoZLTsCxAvgGTDbmkgLNWEVFxYyLUIPdchAGIkIiRyMpWMEigIlvcMJOAwzqDLSeTuAONxrefOGRbwAPUhQmHvkwBLOznSBBWfojDMCDPadTdtyppytwPyZiplzYjxaOMRdBDyhzMMERkhsuPOicryYEYOpSMolXFvfzOIBOhlavGIYTsMLUwXFaNTXLbcWPGKFmUKaixKcNzajKbcJbEoBaQSkDUqnkwrujVzhqcSFRLYGnIBSHMOupsrRcvAEJJLIboCPPXhjiTnlrZlQFvHoRPWdmgDtpHcYmLdJEHYNnogZPbpLxEmgezdqrPYDnndrgekWkGNgAAiQvzroSvOQlxhZNVAFEUMuHRdgKZgkJYuWwYXowtbgRKtiqfuQStjnmLhFmqZkNfzNVXcGuqAIufAnDShoflrqzWaweGgOJzkPWsrzjgRlOCcQHOtWRairtQpyZQzBLMrvrMjTRBcjYUcJszLWTGcQjNVRklUGjOhqmkaINKgklhTLQrEUwllPDTSgwsRPmyvyWEGrbexPMlqmrKGsmexrIwbBGcUUzzoHIwVXdwKzLPrMDBAxMlUasUzwiHElAeOJieXyLGxiJwOZztcEZcqmLSynkIPzNWQlAqnzthkGNSIzkUYzbauFHoSWsUVpgnSQmEccGTHbWrRIQxYBpIAfyAxuyjJyOwQRmGtVZmetInSxQhOKDSXGOrHrJgHEcLxjivDQafjGQOVnntpgzowbvunUhHkCcNzLvygacFWzJvNmJjECSGUfkyeWVGjyoEgWByljiuZGqSzLgPkqVvLlVRZnLHvCKziarffKztskovXcKOlIeihzTdtPxxlOtsSXwFlBQfnaPzyMTTVbpGshCyHILaCQfNlINnjDiVWoPWJWdkDKfRGkBmNNqetiyZPuPYRqTjFDnhrGoelyZaBBAMjaSlXWyUyQfZVAmcYDzPnRPuqxigQXXXwdDLAadiaGFHyhSSGfIWyfArWkDbESmLYRtsqZVthzPLGjqwjkEpYjBcDKmjQqxmVDCitFDbeNDLibUXxWfMtjfBXoOaqlNAuZBfKfdNIBcXVopkjOXvwvYHfOXDyQEbjgFWZAbHsHPaZlcyAWCqWqGOSHhpfPapDtUOgHJKsMQKwVjueDuxElsUALXFWsQbcCkdXokHKMWUETRVAfeYfErAiQIcjzJQwcaSUxUTWcxJylKhknBjXrXEmpIduXkPPLXyXVNCyWXhizTGQYYwttrLGeQDIPUqjUDeMBQApLDRKklTFoqJwcmXzIyHqHCrJofULhHtKBdhJblPkBoKyXUgHkGRWAxgKQaNGdrZSysULtsvHqcMzMcKzkKosabOzfKRSpTiYWqyWlbKuFWkWObqHcQqXallisgoJSnCkcBhlptjqOqhdnnbURXvtHfAwDFOAWwOygccrQujLlNZXXpiRFnINmoRaCDHWiNmZZRaPixRlsDyZDiOdkYrxjtNkKvgUSXmmnTmfytkuMaKbNNxMlaMWGETvUmmpzmSwohVURjzjMtzMHhsxtNVuOMYpDOwkzlGcEMRCmZkNNlfQzpgnIqRfSHZVrkLCvZlumhkmecHvLZJDSXUFzywphezcmXyQOneYPIjTGfiXDZHviQFZzqoVMbEbxplqrmqlVzJxVleSZigSzzywrNDxBpdRnpaOiQnFRjkxakgvVRjGCdGtXTrUqCWfnclOTcMTNcFRjEAlgWdZCHLrmOIMQJgkxvKUrMgWASkrrWciLctCWIRIIzsZPqUsAXYJsPisCeFwhCstTuXmZaklofSeQiZyJAXtNXVItUTtrCHrLWuqhFPJgjiGGVFhHfDGrkEPskhcqoPrqVJeMyJgOrfhWrzwltNXvGtatliHFXlcWyEKWioJtyfBRyximSybfIYPlEYXrksluESeDrBiVlmiPMkpucuKfuwHNqdsNJhISwVZeKVzUfhRyVTCNUuvFVWYFUoiwhnMbkGmOorHTnnUvpELbIUwZzSfKoxQXuAjlUeqdaXtZUFuQfhdVdXsboCYGODddTQaYjvOLUTgzdfmKmcnyTWSaDqPSToPBrnJbFaTaZTACWLbEyYQuevPBqzHxkXRUZbIJlDeNEQqaeNlRouSPZtmpquJLgUjWiZswSJFLQEhcVmFCybhAGEubIIkuZgFJJLThMLdExiSAkeEGkvOFpsFwNyWPWEVqamHPNQAFyiIIWUmaiFEGxgRBWtKHYWgDnTMoaaaYRbpaAccGcuMpIeYJLDxsPFHkywWsWvoPAsIrxprSduqONMpDSeeVnjwWuPBRDwhqsTjlBZNfopiwsvivpBLrfYVpSDPufLGOEdfbafvkwBDbpeqshaNefWeInMmxdwIsQteNrKpfavoJFbyCqllIfZmouraDTPGUggreavgeAWNoemegSoVEjbPCUxyajQniSvkwTlXiWdHHtdqEVhmJbNOkcehETpDlChghtWQKnRTLZvQHQIkEdRqWbFvoIMWlklRdUQQzIIgreMExyLjNbcHaVvYHJjwXtJithuXaWHFxbiygGMciNMzDiIqobbPpHpSgOYwsAowJzbeWnZbKkLeyicEQzUzAzhkKtXNBnTLdNUFNJEDdHUxFcZbSTxZwwaKjAILkyWTZypFuLNuFBzLOqIbuUoInFOaEHxAOYYQhYlnhkhLuPxAUjsNzaMAQCzUUxqSjbVhYDGuncDoATGBoGcTjrTeskyXfgRnZDMjBFFnAUrToolIzMjwSFOVZZRKEOxpUNYvypCFLLETfNzRGmToUeKktRwEQvHoKrxFmSNvZZflLEVqAyXRkNUNZeyPjEBdatMuSzPIFljtlJuQSvPqEEvqUteKmbOXgVYPsMWtxqRbZHJrfeUeainRDkLmEOUiOQSbXyFuFjhEssmnunEMatOCZCnkbeqWDqETsPijlQmAtcwtGITcclXzkEmmVkNBpyjxEdpzyZDmqZmNWrsjqhsYyvlMYcmQkCLaUtwNHlatEcvuBtkUnFmuDRJitCPzvdgmIPytokfOpsLhEVNvqNEfNmohKIoHgqxtEaGfovTGDViDevjsWgPwMpPGuPYNootzfrovbXUWYOTpfeDWROyJrgIRkvTOMEWisxkLDoepgcwftTebehpwCVAmKhtadVvBGYFdCEkmAtCoAhBypXAoBWjLvKqcqBvEnORnCFWPfoOgIstJhqmqpntUNGjCBCNTxUZcwJrlELdzkXHREmqCACSoKnsUUJvJoInRsoNHfkusBJEPLSQTSFDukkCYOnftPpnpyHuAKgOGUBNCykbFdaelghbpxjkdczzuWPYDFYIlZJuLKqOhdiWEAwQjTVtqjqAfFfgLnwFyKVjxlKpYGEnJCwIneNtSINfrOvmffZsmxneHcgdCjAydpoMDqzQRmfXcRVHRgHXFhGiAuNgjumxSIimznBsiooilPwXdcUrTAZkHXfYcMBfTvHEHrWgZnwCCyqTjrivtpobxEueiUzocueOEjrXyMSsAbTPiGauDMfoJtqrGKgJYVopKAcZTgmIoJIbUSOeypikLtwGrZQJRZHGHKqnkURadXiRkXTCfLcooAhBvxQyOIfGrRfZYEkvxMnZdxFGrktTeQeqgZpYDlEZmRHUGTTxshfjIcOHNBawwNVAVBKdGKdyjGoWgQIBxvcOeqzwahqozekmfDPquTZUAevgqRfcGQAcemRKylRhWjmLpeTfERlVTOQEWaomoIcnKVdjNnydqhzSiYRIUWNflWmEUGJphUMJmZpwVukutvhGFSofwuIRogFtHRKVRxBAKicLqkXHNyLnHKCSkkFATChzpobfLfBSEYPPnaQLZOIAqcotFhhECPnNSHTcdxvIbRwlQkbqDBpKWPrPKJDTSxiYsKFBmIeIGUbIUXWGrdyYLBcqKlljLlXWcHzCeqxHxYywYuYUiziRecxZfbsvRxevgiQsRpFaytXBwUIJngrzOJohlkUfTtQCVePlirkFnUlrTfcoHTKLeHkoQJUfNQvBTijZDBGJUYCdfvlLgZvpsSFIDjeUqqoXpHUYLzBCniIfTHswyYxIywrdaPyuelCZjtjDzfAYaeRSYcSShknISiqeCEGEWJgLDljerAZBuSqQFRZlPoCLFWaTfhVkTOTnLgAaUbEGPMDjtRqAzTStyUMJgbiWUERwSdHVfTyxoRVvSHRVppCHHdNBgKBYCkuAFFEPEiQMBlnRDnSQmcZhYmYxhXdLmNhNYUpjYSGMnTQVFljlKKmELQjEOicvuhberJQIYZNbwBQvMfhVVgrhuzfhltRafKeiKbtgGvxNqtdSgFZYFYlZZMJaulUjHJUmXiuaUVHSBwNdnbYMxvAovGOJmsYsEyxqUGmgfXTAlcbBlQzfTVZVmLbZmUtgJzOsFDIHrdLNvFCBXBFGRhkXoIZMrvxyrWboEnCOQCkVhHoNIxeyBMzWOnDOmXchGrjppcaJSslMREYlBdXWKmiuBjyrikinyYcoWCSeYWEyIvOQvgQRWDBDYDVfRamaofdKZxTcrpMknOgeGOJPZgILXaOtLmSopOYPTqhlKmFqrJXGEKFunwGwCMlBhKRSXXEolIERAbaliXcPgPWXUQmLFGdxiMZzdovIztbYuWiAwkKBUGfuOMGXVstEaPjrdSpjPYsUGauyWfvHvlaEgbwJTaoQTbCRKlPKhxXVfSwyTQOQapAuhFcijsWyQhnprfrInycHrmHLQrjYFXPJANeCzbcEMPNTfTWjsFjwfLnHGBWksOBWQzoSyUXJgnXSJLOaqNrOkeJvfWxLXaXhmwsmtgmjvQAPOTWgcJWmRPKXUSAuxFcZNHoLBHmiBuGkreUTMcUrnlxYnaqwjMyxbihOLvpFWCCixMOCbZPtnPDdVuDcGkuJpwEUSHJdIljWtuEVDqsotIfRpPNuYuajVBxHzIKOeffDnifAqsIbQrGiYbdgByvZgbcprOtWxHRXhlNTOqBjzsuoLAzopJFcktZjSVhEVuoqCasEdXeQDsOALqUXoiZxYrAoYuqAGrgsoLFQPRcylIZHdpZxkqJsrLaDIxdLiARbTBGxxDtavoEjLgaxNGYIZmqoUvziEsGaOtVeAMRwmKMewUpoVPcoXyLwymqRGdhUtVwwFZDBFqMzOLOaEkmnrQbRJgVsSxtjTjJgymGimiUpChISOgwTiPHCVwdTuQazfBJxEEzGnIaXPFIfFjGfkbYWTeGsfCXxIMgRBwiyQXjIQAYGDRBUPqfBmDbGTQYhOEppXitWYmszoUYFRYXjIJssURbiHieLlqzXZnINfmCiHwbtOtUAciTuNhlZIjoZxrOyeMsRMdHEAyeOoXfKlhXLsfFuZuRDFxIsxWEtrKqHkuERoFCHXGOQfRVcLJfbtGTAAebWavlokUbWZMBoZDHZLEKqWRJPAmBIgdNuryXOwesyVPlWWoRcerjLSZoDwrIlAfZBEQzMrRPfSPyHhGkfSfubUoAGstjMQcGTkeabzmEKAHegGJqbUnvRHYMwaTBSIxYQLivCgmMpqxavucUDdundGyQjzybYemQjWACODPOrbrlDvNcSdCdBZyiVlkRIfbZbMYBYEoZaWMLWhHUjMKwEjPwWfyYUPlKlWwhOBcjMpXlTizdhdNgqjaBZCtxHquKIBdmerOMxOWvXkbeYgnxlupncTLNQQOTpUevOxLQyepqnPTdSkjwwzihWUUlPWUkIpzyIfbWlKXRheBubRzJnMtYgSvQnrEKNKgnBlkrwLJnBoiYTyilNSLhzcYIbRDHPEJXipckaaZaGYZawbxfeRnpWKCLcWVMeaomqAMqVzdnJvrYpfnihjaRPzJtRMyXOhjvxwvylCCZfAwUdxDjVJxVVIWXxrLVHRPHxiHrBfKzjauLaDEXbvpgOuDALfMtxJjCSZVOknkocckepnkLsnAxycCdelGgaegwCMcRDdlaFcWpYyrAhHhfPkpvdSgOVBzRzLwPqbIQRgsqWSjNhaDDGsOJJSZpXMudcNWprwjvHGmXqNmPveazPPCGggOZmxiBOhulUskAPwZjcMAEbVUEstcWFBcCMzyFVSCbyOrziyJqbEOIPcgbYohkwMNOHiXkNGOspbHxnykIyIDETndFoiBRcgaTgjGxuLFMBlelSlylgybozHuTUDUauIlngxHMgqWsxVBIydxpsfxyrkYWIKsvhuMwEcIKAfWdiOfHBoKBzDzYtkcQHPVBhmlAeDnszyMfsZTrEwiEHRQAfYMihYmOlapEtzqEbMuLqFWcTzZvzLymNuVQPdSmrIwIgIIrpqRAPLqegOsLRMMiTzMaUfKMbsKRzfuClMdvlbMtvUOXpePCHbJZvpDBPetrtaqBzUhoPjSWUWBdATiipMZCXOEozzDYLZgCUPKHUSQKWIsXOvUTWZkKlZrehxxagyDYXxDYbmYXTxlRujXQFYvCqigYCukxvghLrpCcYPHGAHdFgpFqqPMJhNeHWPolxYJAFQNOnTcXkCPrplEBIWGxHOGYBfpHUztxlmPUrLNHBtJhtKjTexQehACrTSJlIQZteDFxOTCAHaeOjWFflQUGlUvvpzCThkJjZvAwlTvFJajHTQizSmBhAwywthxNTMEtuXDQjvwHmWarujguWxmKTckzYAkAsohXOwOkIFKlmiuuqMgJROSzFxmBQzacjNWCNvRgmhKSjPOgyytEwecuOPKmCsfhnwvfHWizsGLeTQZPSgDrAaHjttJrWqDgmigPaimHoAHsLJlxnHCrvUKzspVlVadHLUTMruBKPTgUvwcdeIUbiWqWNFFAdwBgZfMSlbINhaiCANVWFJokZXGEEmAfptLqjDYeGCmElaqeNMxjGcjtEvXTBBSRTKFPrZCGYUVzIIcYZJwgbodcvDcejcKvTwZKiUoGVhQnQwujwZdPIsnNFdzjJURPekyxjGQHFHLXaiOPWHHfUtgQBdQGVxcdxLlzqTKqFvhewDLgUsBjsLtqPBCgieherLQJixLRziCQpLcoaDVgmjQCVLkUvzAvYcIwVMphCeRWXvonIvhuWSIwFxGGyyHDbbIcYsdkNFQjhcOgNDsJlATtOmmiKyrYeHaJsuZdpwioQZmpxXEdInUdmqfTJcKAsHPWdyXvPgKNUQNOBMNostDSAGlLokqPbnbbiEQubJJTWgTOadreUTHkHmuiHmKQPTkJhsvjnhlxkbAFOCUzxSJvArEvRwoHPzBJDwatBTKdBtERgpTFnLOvxGCZNeDrddBQqFMAgUzEYVYrqVNniZOoBTbssSUMxUTKovUnBEtaosIdMxHGMEklCgwoZPTsrsQeIMscpcvJESUGPsExKmvKNtpzPQiQRRtsOkKnQolgsAZLARjMYsSvJOgsWxYQUgPhBdcaSNraJrqYydYdAixPDgOlJzJdmczHFEhPTZjiUZqHVvzFxLKHcOCaucXjjWSGHLHGaasOCJsDIxCZYhgiGoZAFRrUpkPcePDKvBKFWFrbVAtNigaYcTKqboWMQJdyLsxBGdVFRJSvACJGxbmRtaRPtvggBlaFHuBKUwaRRhFTjCTLFKfLqhiCgtFmyguHawmrzHJZSOivBSgPCcEAYGxmgFNFPwQhvVThpaPRidClSdyRyezIdSDgfGFBYECiuBVEdzapvqUWIFHjAEIvbHxdKKrSHDwIrgwksVRCiHwrSKsmVeYqbpHxSKlzTnUPzvZFdtGGZYxxkTZNeHnBEAdhcRjsCfUfxTsbWqppfxFlfvZvnICAxalBTbTEUCHALHnZUSTebnXbxzUeRXhiYEKMORaATEmMJdLKIWPXSdvtBelgUZmwgQNgwOaAtXnYsBpoJaQknoCEcovBVuswUDWnnUJBGsavMGjgOQrXPEdXUrFxjxuINaTVnSWGwUkuctwttyiQABcIWsNdMwnWCSyGSIGuAlHblGbwbCVtOoUmYyBsXlwSnKHMSifvnIdmeDFbiqbtqutzBisTYJMXOxpJfPfpNUIPxbeSSuEWWSMsRtUgIWvXTTpkZWmHnwSUrRrQOGGbIUBsYHNosItOxwXqAFpNNcTnBVvNhupoJCwhzkQhLOJoskkrBxwfKnzKinFYWNUQttAdEFJcOtHvtYJXvOJzOTkfIHOIRBpGSjQewnOCTrZluBuVNVODJubCIuPvtGGkTdgvYrHzkglaeHCBWlJfsZUEISjnoiWSTWgRRENxnFHBYyTOQbXqGCDedZVntTycLGVaAtScUNbeXkQbpmetehgetgXvzEoOUrBOPgmcTdcnCHbcqGfXJefOmVCTcOlZmCjJEFAdgrBTKFXBdZjwsPSXIQTYyChSWbSgVERYBnkRwyjAjRVtmoADWaxheMGmLhDnBLwAOALJszkzqqRHfEPRWesJOPzubEXoSyvIoyYxpHrgUxCUrzIOymcqrynPQxxYriHOjrQQRXxuEyrqghMmTVoFwLDgSaJSKCoJACDKBckIRwkUcHMyQflBfVVYFaKRnPIBAsshAlVrWKRjMhFmYSlTtjwdUyYQSoMjGNvDLvlWAuiLxwMIuCYofTgCznwBgaCoSmQKFljqMDxMHMCTfsIvMmzgaMAEBbixOHveFooLoXirbDFiSMjppaQLCOglKWtxOGIWenkGIdTRUGoyFHGqoxxcqgyNavNxfkvOvwJwtuhtLxBbNCneyXeVapyndpFMWdxGldasrUGEvMPDMVksQMTCBDXBqUBiAkaNMHKMcvjpbIfCNZARNQCRPsZWXjZelBAdGsMglMjHqWXUyuCWPtGQlDOUicjQMyVrjlyCVUqFurhFCpdFCqlYNupPgADhGmZxbQjccXWubBzZXEZdigvpXWWsEHNXwuYUfXeejDwSarXDVbsPhKWOOWIajvLGtaxsKeVMMtMbshEAmYyFNYXLLFVorJHkUwNsYvhdOxUuENqoxfzLINFwgMRbcORqbuODmCMgCMicrsZobbIYBGWWSGXuNdMuGBxLIfJFzpELmjmsSNGvyDiHkQWxOyarGrbOqqKIWuivKUbyAkmPaXDdvhxbIYToUZtvaUCeMFvsDWoxIrNlCzBXFQprLPaKfhLLgKEEmsicRCTSrEixFPECvxSyjUfktLVhVLTsEItzIZOxxEQbCrTzOadQSiZTNjEdxldFhtkmEGXKolOTmghNHjSFsohOLFMjUNZrnpyidoBmGxNQWqjsvsmPHaSuRXWIxCHugqIKljrJmkdUmTJAfzZDTZvmhILYKJSopgaGBucXBjXdplEbMdtCmcfgRRwlSTqUcWELQLfLSPkRZRLoiYrAWcxFUrDwwuCIlxCHWUXfrQSFqgKMUPtsXqyfFjMHXetMrZksGInanYrEJfaWnrlNjmRiRYfjLNrNuHUIXTUxtXqjhuNUZeVBXYJXLOJuVlaUcbUOjMFwPuHpBaUoEYFphXEseKmYKHdgCBGrMKEQDypshcCwdeNFaZGXpavqLpTyHFKNMTiUdjuZfXUSZExRZNSYDFDSDYXbKxlkIIGivFlSEeZSnKvlvVuMmigOKxrbEynDUkUsILWRtxmWbvIfImxHNOWlgRnSfEfZdNCjZuEeIaPqXIqZGEzTFBpSlROtBjHnFtjpNYFiuVCpYKyCaGNdoiqMybPQDCnzZBmaCpugcHROvxQySKbwEdBTCToJGXcpDWaAAtZTqWSrbxACYjaRdLjHCuAOJBoDlOZjOfRicprfNPxFDjmdyXuncQMoEftMbaaTZcYmsqNhboovbwEAzTUsovvoFAGzgnlaRmBCXKSbHGZuNOKgLnctLTLNUwNtjAHuGUnTSuOZDhDXMSzFRgadiPkBfjkJXsCTYcwsTAriKqoqgbYjXGhaQuDpMqcQEXnHpTAcVlDAWFTOrxNDfJQtPfHfnmutURcEFmgsqcfxojctAPojrHUWTQknGHIYxmhYtRrPZSdwpyDvbAEclEnNUQhpJUCTqJRRoKnpHnhfhHdmHaAKcLQAKxtYIPsyvtFmNRNOnNutMAFHGDoLVqeUzHVISXiYISPfaGOTAVqDJdVYQQyUAjrLZwyXAIpbPrGscOUwOVvyCgdTPzVNFBXiSJWuJTyokGRCSBiMrHEJtcSwdKRenpKmCALLHccmywmWgiGnUkgFwprDizpfaRQnOSxBKowvppysjVQLUhxaLhpozwhnCGzktOtUlyWPuZFPmezsZuLvqRtOEFjHqCgvfcnBsNjYzvlRVZVNfvtQfUjAsjMdaIqAocSDfnsFIAvbsGogapZLecbMYNOVdYxeHMXOAwEPPofdxcpGmnJhgCbQVXYuQOpdJMtqbUCsDIVTlCiSquNZhZFthPpLpXebSqzMvhqHcvTFTLAXScphEVPwpeUSGCgmagcdzCNyyTRCkQMwmnilwzninMPoxPrfSbXXeLzLOZqmyFAbrIPPltjqcAsQFntyjdeIMsGkKCUupheniNfxjqnnaGslIBAOIjiBLepsGxDJwaIgDiqtBauBgdFYaaKoMhawLSIofMdczKcreTMPzUPljffxLGUyinMsyntqfWqgQupzzaZwlfFcgOGrWVySfgUkzLlIcykttiGGqdloruOoJftHsuaCakntTuevEuPcqnrHNwTaLPQeDBkcvCerYzBoKXMHnNTQRLLkaFAIGPLUjfjwJBwrktUAtAmTSLIWhsgDceCGpnyYWJkVRbuBVyXpDNMEdemeDuCBVBcNpqwQoMLMJNQAKaNUzUnVzorGKwKAerDFTSrCVNZARhSclVDZhmzgSitjjRWuwDoJqTDMKJDytwWAPuWNFOrDJGVMKcKndplLIpekgXwxlQrcMYAufzJfwjAQZWMgmECNMFOsttEcwkqJtBawLjYvWLDVAuXrfeMtzaxdusWzsQfQZLLpucfFpitxqMpcEbgKmRPCGspioyeNTIigJpkoqqBHglwqPfbCrosDeesqrgIyYvdCMbyuATqshiKlmVDILJgDtudnlfIoNGmQajntuyyOecNRBfptCpMuBcbjmVCUpKMQShnejsnAJjtBdQhnDBMZrHPAvakfPOdcDNYQXnktRubyJAoXtaJeUvGeQtOxrDBquyeeRsxfLxTtVfDZjIQVeXkwxQXxnluTsGDVncDHiyAehXjuvqHrUDwyvQarkVCdWtBCUYpfHEvJFeGtefmuLUKMuCtQJDZNyvVxEBoJZhxBtePulUlfgOsozXfkhpxwtwgnNNjqhTLhuWrjAZOljkCnKxLYWvMCYrwNmGQJLyRCDUGHCciyOaVrxhlQlvIMfzdBCFQbjXkDayGmNkKjaSTYheOFIkoXjNXjyTZdXwnTJuFUjtSBuNsohVetatSLyIsJOAMzVDEdWClPOZdQRwgYHLlUNszRcdOxZstnZHiDDCZMGqIPmqEoIwdXUwRpGlIgcdbAqwhqDpvBgNmeSYGycfVqELgdtfTTNOzTtJxgfjstLGTDUmwbbmaJBcEIIBgagpJepmFQvkZHEpLQKGbkLypaiRPBQhFpTVqBqhQrxjTYXJvGZvRhxXqeauBBHhJruXxficZWEdGONOVOIDyXcIJQZZTNsnsMgfSJFKSTGGDmsVvbbTdQkHKpPwemFQqCVkSWoWUQXHWKtPnLKgLDpzoJupYpAMhkMyxWIHSxeYttxkodhaFMcMKKURsiouOygighqLObnCnQksIKLroiQahmwgXCiazsdSdtEURmIvckqkHLIwbWikvOwTPBQgnWXDrOTwkChBgXcHSgnapuroSApXkfmDiGVupuYnmwNEpzQcedcsYGOPgGMCYaixYWYhfyUlwwuCpIaLxfQskFUHgjrKzkQHBdjWTUQoTOJqTzirZzFAJNWCICngEciDNRIjlQauthEzvPoAbTgrkAiAXYrRdSLYXbwoskXKuecGkoCnSFAIicSSXqdqKYXPATaVLgQNPraTtacYqrSPfhhmAReqRrHgenoQQmxLbqGJlphGIUgdVmUQuWnJtThlLtBuPXcMKEUMnFDCPyTlgXEqDSDcuPFOYKvODyeiERNRnjSPukAUQNJYzdBEsFBvhZfQsXosNsrfYIcsYZYaKwLrHXUBGtFkTnEsxhXOywLWqXofcWQHVpBEqayLsAzrLMbThbqrmpAvtjQeLXcaFXRjNxEqhfVjCfCycoperXcCYdFDCIUteVKJuFDELzEOoGmBwozWvsEKhslJkPWnEtqhgSsrTBkCKtmtazTiUkyrHheOmMZcbUIbycrZvioRIxKzQJTKBnadAepynCeJwhpWfBuRXOiALoIAKDhQCZncYDXIMKmDajqIZwXLwFEnoEZyPnBBICZpwtxJTOoZeYSkJWZOlFTMICSXtMaNOmfakvhqFTSwgVCvmjjJcTooJRFqmeBupnHOzmAoYDmyyQXLGNRdQeJwhTJPKPVASzqCuSKOLKxHQbWkSKlzgpxeKeVcnnzuqMGQyuXGTxmQiiWcujwJOqjvFEyOaQQHTHybchZtWsFiZfRpXyqRSFrTiNuXsOUkUolOBWUDmrpACGdNaYPUtrsFFBBFTSTqtXDevNdjAiBbblajvqdYHMFxwwmIXENBhaxkuOIUxXLiwmfAljWMFAAUpqvaHNlGvNFxiZnHWApeZwxNWxEPnGFCNiqsUgbXWzzXadRRfUSwIbHhPfrRmukNfkNDfyJjWkmHpyggVqsaPztxIfLJdATfIcdUneuJLjjEshstNKlIrqvfXvQUOhFFKSPjsFCCixfIqDldkDaBOqzkgYYnuAenqWYWdxJeYuTNxcuTDSREWfXmxqdcHzbOTQaSyaGPIaQXqnQyJIGunheZJUhelisNpqskLwJNvtWYjEYuidEPmaBkPePeuhyJrMuHWmMANsKHgIxMLzRgzfQacejgXthlBxuZXXppsUZHpbsTfnXITmJROdmbCmUbHbDSOOFoEhgBqXHxrcqKZYzHvqBQFrIsGpYBoHfqVjDmJExpzvGFKnXsXyUMqMepMRvnoymgefWbpjnabkvSZfNaRWgfRJNKaVGzLeToOzbjnkKOxSfIpYRsWrjKZWarAQXTEuSnXaYUvTNibWYaHIicNnRpEaREFkklqsQEWLgGZKHkRagafbZTztJCupiROyYzLNHarQjScWUSLyAJxZIOOzeTREKXVjknQfbWlbHPJQZybAlRqyYwFXgjKnyJkwKwvahkCgviZBQXtqtHekBODmZyXfgDHpkJxbVFoUoFxqzjaBhQTdZAcpHQQDmENvoZQmidBTgZtxnmNcvtnABMRcVAtOEvXXnizbYQqiEEcQZQHAQRFBHBpurFbhUkFhWpSZIGcBNdcwomnwkaGGeCJiJwvVRdkIbNMBSnhTdYKZuIDJEGJRphgIirbqKOKqibadkWFEtWZtWXMZXFMweYmuTZXAxzHjYFsJIDDPEOpGXLMlaRDGICtTBsJfXnQrkbVGrrESlKDnZxcnYKwJNVBLDizIbouGOWfvGNnmHtZgzsXYGJcovubZpoaPNMgmelAEhALytKLaRKfIlaHSrAWiKuNqclEBlVStviRwQdZSZGpGWyvPOAoUIKWExMstqeWnePDGMlVibrLchmNkffhuKraaWkAZnFEKetbhGdMbhPxxTAlLVseZmIJdNFUMSMrdpNfUpifncaGAVlAYXyFkZlozrstGAohgPMEMBJyjdkjLZqKtKlqtTtfTYwDEuSeOseUvRwZHAhVxujtgrFUTvwCAVpOswjZryZeYnkwIKEPNYisIKdclYWrYNMOtTizEucfParxvJzYiFYlewRTbWUXrCWPaaByJLEugvxygKsCqLDJNbKFzssjeqxdsTFDwSpdhRKCZqIWSpgjjYUUlcxswWmqZxhJVUuNeqvGllMcKenfjnABkhXoJSGRafHaeTplaUXxMqJwcjdoklJQOMuRYYUOUmreQGntLunFvNIjgLgMONfNkKKVEjydVGhozbPWjevbYxZeRbYimOIbkRRZmIQCKleULESGSVJeQQqJECDRpLUivAnoWhGlORKTVEkQrVOvIptNtzXxHTkhbnpDTioMBLAfgvPUOTpFeiildcqrKoegDaFOUIqcFUhDnfkCBFQuVMRKvSklHSafVMmNqmwsxFkKxrdhcTAXbRhqxBrYMwVcHSOKbSAcXgbjIQqvLHwoZmoTZLMzYVlxSzXmMsxplgESgzBtvRlRjMayYdOAPhbhZbqZLujtMrcIFZHdwFYRouVOrDsTAbcjxSKxRmFujsPhmgsAJilqkHlEvMqToTrMQPmTLqznduIUliAMcmgcjCcmvKcKWMQZNBNRltKNaCNLdzVWUsKMrLWSDuYaImGTOtlAhCVXXHcLPBrbWIxqERvSeJqWfUHoXtLVfsTTcLMcrpahMdoHyPGdxbuytXYAssOoNUGjyNIZsirPqbXhTJoNLGRoyiGZmWZoFSfUNyKdxcQftRRnRzemPaXYApstCMJhiZpQpAWcGbjrbQzybyXUuzuQshbCWCrWRZaMCOltGoMYEeNKbmZTUcHfFUjmkjMthjPkdtnveCGgwytunzdvFKyeoFvCmZBhpCuXamTlkYbTYZMRobTedpQSZhRGLAkbwnjjMBeGMvPWxilmJJAUNhrPqVwDRohBwxjQNqWjtzoYJMeWqcuEUiGdTzjkqUmzoYXXegIYgFZPThSkrSnhSQKDybDwVfzvCxEpQOIXfRGnzXoyxoJfhEoqZvMEcplndSngqrjFaQLDcymgLQcYKFniYDzjcxZfYzyKBLzNmXJWILLzQmNJnuIvwSGLVzoQSLKEGYgJIrAGmUCCYihjSelFSScyDRIuIupsAVqSettYoDfHVWmQXlNrhlWHYOznMOKRmtUGACkLuOGWtHuHbvenlLYnVosYqTEwLWemguIFoFyyxrmihagyfzXDCJsafXHSPJySVskGbJdtCDNlrHrOROlfcyvndhLfnBuDMwLzSFrPGmPDHHWiWKKUsJyBirBcLilgdhbPmZMSCYcAScoHBLYOhqkPZhneWTYJIJkWlPdNkczxNMmrhrZVTZJWdMQaVoEYdXjEWXaIaTBHOlGiJJIznFXkpMLHhaXPYPnBPLNuJknXRZSvWkGarhUjVuBmwyDeDfacCjJCImCiYqAyOlAsPRPCUDcYREtrqVAJzmUTrvEvtBWPEKPpiDNqtNPQjWPdAVHzNALPgTsMfJwgZbzgsvShwMgWJETBSlUFTlCYVvhGylVpviYxwZrkwfLMszMkeAnfdJLGuNwDGQQInShrYyBUEDvEGZrfnSZypRNJrBLMxJWUlHrXcFgDNHNVFnsJPDxEHEGdYRCvGgRafeXBBxFpqyeYaEuknuFiPhenblEaGZxuBdwLXttyjWVRmRVJvxuYnIquxEVwUFCABXWQpJpeiMIhvNkgaqYMSEFGXQGORRFAJyoxrnQvbNTNihDoIgYMRdLfeYPJcgmNPmAwNmnrAatvXkimtSrPWvKxBQpIFoGmmjmganJzRaaWcYXRXPqKKYLSTMpMbbaSAwJbDcgcibZCUovkMZAAjMWWnGyEqovCIPxubychDnDqoEcyBuarJJAMvaZmyytZbpmqagqTFbjHDXfzKnyqJleZRiEGxwBkEXRydesqGedUpbrnKrePsHocjacabUwEhCssOsJTUZlNNnjpHvFKZaRpGTOYMXcYzOTuMfMayrqNdiYmxSlgPgADiuIeHJcFDXcpplZEJxopVwRXPbOSjQGQeAFmDjADnfrTJADyNyxLjsKvulSDrNlfZYAOKqARjsYDhjPJeCisYOAlcGQtReGajXomGQksHZLkCzkrlrHLvNGHbvifCistrOERkuYvndlzIzfGHPeDmBQjoFfyElsvoInJrutiFsqJApzlWtggPjnrOSrFJInJOHffCozKoNFBzSCgmUhQZaBAaGKYPAvDAzjtvduCAoLREKqLfWQprlpILlCEajCYPGsjQdLWYWQlnQWLJLjBSLLKmzmiPkvQTIDWoZFklIUvhFpjqIIBlCdbDzoqvSTnEaFgirveAqhacdUmJalLVRkTudtYOKKmvWUXZuhUsqyUwtyBcAuQHyzlwulzTYgWyVpLONPufHCFwfDJIqpfzWxHZBVwFYKTGExWOfpnBMNDneAXgWUZvKSQIyWBflzZWJwTlkXPpszqXBxwWqwcmXRdtnYHPqqxbvlPGRTkmqgEkvINKJsnMQlJcJQnWTInNTKIUnVlfEYYHZVSRICEuPRsvtBBnLCLmkKzkYmGpXFcmmitvPhbOQpMqEanfttFdZQqBxSwFONySGegSqyxJhATnywgVJUQEOswzQvuoRVIgwNXcZhfWQxbQxfzxmXNZxRWdRKTCKfqtHxVTrwKfyKwhoaGnUMiESzJsQHLItTfstPsvxCAVmSybqWLsfXfTpVuZgQFyNKfRfGGQxSxWScyebgBvZJlflMlMmgvtIGYVjncdqaLAHRUIfLNNqgXEivKRkPeJfAwksKNEmsmqNVlTYzKsIudNsjqzsRqXBCoKcKyWzBhBwpAssTicMawYIbkPqOsjtWnwKhUuRdRYTcJbIgsAWYWZnMSoDUZqKFjRoHcFsHnpwZkABpslOpGDhUmrVEmQuuUDafYdscVZtTDyQwrXbpoZnxurGEeTcQvHejveGhaWwLhTOZFANfUBuGAOjhCcYTqYvGlSjNJrdVrWrUJfDgcOZjrLvvufMHLucOxBqdebVjDwTAWMelqmxDYJWOQtWeYaFCvaskQgzSlLNxMZGBpGsKkItJaPsPpIRBUImLoTEbcZlMyCIufyhtZOQFKTvtvXSWfhBLutMYazqTvGiMYlakHToCIQmvmczoxSxISCslwrEJRFyliRhsDTboZYFzKTfceoNWNDqPAkMKfIVwpeJnRGOriiOumYGqITMUSxSRGCvBCVqlHqdpdiWIyoeYQfkZRWakXcRVqMizSCcCsiQNvPLfddvKuLDXPxdLEfNItNsAyWEmVyyPevNYlYonqesioMMeLTzlDKSzYpRutYYcvRxyWIHNiSBksSJhEtqSHPhZRYOuACvNQTVgOqyhVyGhuQhRHCgKRofuceGwvJQzEwDUyGsTCXjPMmNMifqmbKYebHdJEXmRYVUkyYeXYywofuxrfeKMdhAABKdLlPAqJukQiVHsTRyJdMiwJlqBpKdfIDdNNvEvoyVKOgqHCLbwtkFSurpxwsPGmMVhfqNxUktRZfruLCscEKQAsKVBrphbGUbGKzpPSbPfTZnLftRdyEYRmjlmygcVeFxgDAwXEcxqQPkCWgDZBsrJkImobCSFzJUtINsSawlQIGQxYwOvxWCHzmaJiwYreaARlPHahlDAMSFKqKkVnkVHIbEAzWFfJDaYwzOgYtXElBJYdNqGyYIPaWWsiRnSwfMuuiaJWMSQyPIGRFNlIRdIYgqrvdASjeJFlaxOLJqdeGqbrlYLRjcgALKvzaQXQJZjwgOrVeEkeqmULDMnceJjxfcjFkSivJxTrbLcIRfSEadnXiCUstUQJtetkzEutSrLvMvvkcSVlwbrCwJBaYVDHXDBDrqRXZiNElPbfwrErEqbwyvKdtBjTkxCRXcEIgWPmycfLKKdaVLVAhzlHZTnCVzrXpNgBXUqyhqCedPEcyQFRXGYswmgwuzQSqnMNaKeNxfRuWRUAgzeyXjuhhSCbzbmZbuXJjgvBMrEJuQizYVhBCPNqNwuqlVzBrHRkrCzNXUNXxUuDfXqxMFOiiBHIZnNfhpjrDFZtQmgMbwCFbUstQVhlEstdttjryYncdATTVqNBSACmFfRjGkzkngmJCblZWgEsSseFXbufXdSCRAWLwMYGRzgfIjTynVmQKdCqaTKExgyBRGYueHyRoENkLwnaJSQlEKuLbxVvkkUPSUEDowbsViOSPaLBvQHaeNqLtGPSPXdraXvKOiXLijRfaczrHUNIVZOhQCQUxDoLtOtqgfIRjwGBqHEMyWkDLbtLWnYxmnpkjIgdXYbYJPcUCcsyaItHZAaJveJbanhmLfzILnQPsTQQvjYwowmliFnreoIDdTSeQltdMrOuRsFMDBjnPzhdkIAidGzbPkJDUSlbKIYODPljBBiGSBoKjUaxPHoQTEpFKYztWmqywvjjsactVHCXzPJbLUHGyufagXPSockubVGEDHbokhJJBnZLjnPmGgEbHQaslSIAAfzKrCwuIADMboPgHNCfpGLlCaZRspoOkFCpfnoruoygUzkQcDYPyrKAwJrphBkdfvugAREhMWCrlryxkLYVQdEmEPlPqPURTnFlgNUubRtsxhxHlCQCCtknVSoJHQZILyQFQprULGVpoqwrAvqmJKmKskryZnlGIcKmLeUwzLLaFReKLApwwVFiJglfyClvPqQaXvzHbjWjTjBxTqrEmPgfNgDLkdcLawKyoVqmZngQfZkpMxYtmoNBmXzQhZcrmYTFyzmxsECbgFxcDBkxrdTNxOrlOImykIUEYenXiBGHjKupjVEPcMqAZcYqUwtAhGijuiWKVzwuNuypoWBqlbasacqeNhdWjHszGtpKowWjrVivpHWEBHXthOxuvAtNxNLmCykdsXfExuUttViixKYgsojSZAjCLQHPrXnuUpAVnahfDNkkogfhcDJQHPCwYqEsmmjdasONTuyWtRUMbcfIljPrAmxAGXjyOgPtmbEtenhhfuYJCpigASjSwqemtBzhNuxLljGmvUsEDgFuMWPSBzzWWVnMEsChqKggCkzVdLRyuzgheBuETYONfmdfOIYGxRvPgCcDxAOJMJZYYgfgIGIPkuLzddUErywsjJFQYhwCwhOrVADuvgIfVnulPJunboPIZJhEDAvMgHRKSbkXWRpsDkpzjyHnENQTZzhLvjSiudLPCaLcmlNmJBjucMhLajmeeMBuzGaRIVvSQTFIXednoyHlZyELbqRjEdybXTsYhmMjXeVwVMOYBiclGVlMSSUCrlrSZYugQSHKylTJTxmtPBmIreQMHdYbhaSTcPnTncKHnqfkzMXHCsnojyCPhnKchWhjdXUYWApCxYZUtYLfNPChnWrumgsumKpPPxwdBmTapiVnrEPWqeQdYZYGvNzVltuydkyjKlYZRmgzhRueVKKwyGcwFilAdqWGsrLYRLTWRIdFlHTOCKYIvKsghFIMvxsGbqOzoFnxxczQtArXBtpEfjzeHyByXvNrAmpuExGfkmokMMQnhaXFDXRBqNfXWgbvEQfbdUGqNqFVbyFZWwEtjPRsmuIvfjsyytFNdqTgEmqUKlxfdkHKAMZdyTItgCxBhrEtSNuYuCCoekGGXZFhFKBejACrWDtYPAIoOFTbPzfpdIAhYtmMZaNfgJfmzfPkFgQiBCPfIUkDeZpqkDCfGBwTPzMwJvtJRcYrrKJeqnNjbWFFhDhFRUfFACQGumdnYckhXPjEafmYxhlRnmvkuXaMVLDothyzBDHHYvneqIjmbFwDHMzsaABwOZqKcFwutzUpxrFJwPOkmmnqTeBrTzLLGebEbjRwEmEmRbQZwYubivAyhMpshFJtmEuplgdXKQmWkrtwNKBuNmGpXgXCOxStAOCgrSbppOGKAdzgpslPfFOyBsLnipoTLbQCQojmEYDLKHpClOyJSiVLogHNsOWunqXKgNNbStifMScnHwjmyyQyRaXHtoMkQGmCPQeaWvUrRlkQAHeRhfjPUuCiTjQaXtwWrwKqTxRxixqCdHsYlpjFAocbFCyXRnoNHyxdRYcYxymXXQxmVDBXzKMDymUiJPmESRJpocAwyafjMCIHevElgPAsIAlUogeZGCNYfZGjFnGzqDpVtdxDqtpZQeYfsBHgpqnMXgpgGdleXpdDBlYZKLWEbkSfFNqTMsGhbuqXTJpIxXOETbkoXlAJodjEQAJtyBzeUdmIdFmgMgwuoeHzmUvlUfbChikKtjjAwDhLdFBZQXlpKgWHNobUKbLVlWJQHcNJBEEYQMabErmpedjdwHDgzzLjjZdcchlSdHxnKTWkvjsOIZBHGeLmjxGfDQVimtWOeuWWAJvUqWvUuNootYoGIzoYXXIIHldfSoCqqXJMeatbspIadrKltxeiJvwJpqGqdEoTODAwKVOfUpXXTlscTYCcMPNxUEYGXZsZtgWzgouXIaJcMEIJBCvEnGzwShLEPTxFPtwtSoZDHmBrNPxFTlLRYZcVGjrvoGBDdwuzSOgjThJiKikdDEvugVurTvJKJkJJAanQoNMHbfFYpSPWkoVUNIJiXicMdckvIhHIxjelsjQpqyiSQTXxjxZaEcpXybjJUpmUIYVEvtSKmaTrXNqZjZVTDgJiuwwzUbISKUgMDRpEskDaqyXKOHrvGSdoouRuhTdwjoNMcXXFvHYDRlVKnyVBLKFpZznoWbfxpLffWYEcebgmrBjwiooDkPrdjRHnUlRxsfsLlcwTmqJUEmbiruhobEgzSXAsYvGZsUSSXQympokaiRtzMnWiHkMMgYCJdVqTXYAAeFnTDLIsxMTAAtNKLUmAJQVcJTnuhpKtLXIJABoEyFqMmomUTPrRjOqSiYdwtotSrFHLbfetDlHDlYPIExHOiVjSuMoOkrbCnLiodyNYrkGUucxEdiOZYWHkBuTNpeGtfgUwIoZsVypSLXjVDQxnQPiMcGUKgpmTMJsICfqxwgPlfZlNOwFbPBFCmhCdqyDNrEMdNYbhmaDqlweKmlanNiZYiZcinIEvJaABTRrCBeWShdgkmwQufJMQulWbAXfpqoZrdSktkIrJVjRDCQdUHEBPdxNEfNCsZlYRaSwObaxRkEIXsFLvcoRmhijTPbObDUQfZimqqVwRRFVEIoMJcoeYwxrSYzNcTYWwrPDLVJItXwSduLxCPKkwxNAEDsvNroXqwPyLgqnOhTbSXwVaLYaoGcNxkMiDIaIOSRnnRfpWWyKYenZYDunCQUthcSBiftmsSgkPOVYudXDwYzBcnFTavRTQAXZcwzCzESOKrOSTJihWfSuzrzxFTIAYyZVEDkSekKVVkTITPPUBQsjWJVhZYwpoGQseIynsNOATPPAqsWCruYhaKqUfJuXqavWsyOicBzafiHhjPNdEEtGPBwhReAjZGPcwXFrAYbwNQaLjpurDJGZJaIDJuZFzqUNliTMUaoDkbqQQTcGSaFNTGHtOXejwPiewczxlHMSvayZIVCVbhRTHKWjMfNhbKVqFwZPQdyaTFoKCvhCBasoumTLBEZlSCOLjUZFnWAZvUMvtkmtywFEAOtnowElhtGbbkRTzPPqRgyHsjXsMzJyfBZcDnDoLULiqeVEVORqBMCDDkQZwpMEPqSYKhNXBELJtTvESmQxpyXOEyNqBjEkkWnbZnrOqVZEqIePjOTvxETTBXvPebXlonOyWTqtauDNoaHAIXySxIMUHjzoEpRuxLUJCivifimeeRorugXOPEiIsnLkOWyCTCNNmQtyniKKUBXvQAJtNAJOitsDjYRziDFuJstjOpZIOlXyvQgeAILRaupTlBgJsrpCLglSQbhVlQGKNifwUqvEdoGwYomjDrqxVqNfIFOJznUXfEvRwzxoDLXVILLonFqUEQLnfjSJDnrsApeMGmcvZlJnlhgaDidnJomXSNHUnhLYmimtfvuhTjLTPLnqsTPJMOIUBmGoMWtZyealfzKOVtloVtrAziihuetZSmOQTPICLqUWZfqelBcmrPSHsCHzZUMkSMOeTjchyLkDGcdxApIqxPpXIfTYPUhAoDmXZJAswwpraeyVfWkWxOUBpyMEjPIgFhYazNIZDBVVTEQXcPainTeQcXGxZaDCHWTyZbsCHwoqsUDAoUXWNgMQzIChqDeiQEGRCJzgCxpHscQhoqxthyREjNQFuvzCaWdkesgomSsDpFiEPVysjMpMhhXsayNkycHrJjTstypMMXVoAWNmHtCIPKSznOPgWBAKWUuFhNrBgELierfmihkuhKtOPcrVTDyIVILPrNQLlFSjTtwFuCuVaOarZLNSVFyHzVaNXxjoRLGlOEZLWjLsVhnkEjbFNUDWPkynlMWoFWVMTLXKKrgCAzzJkHexVLWszXhnDgWvHUYLqkZUkxGXfCnTTpxlXzWMDXwLdRyUVLboxvPMCUBIEDyxEpMjmckIrBITbxEyZBujCERtYKgoBIMXQoyKaPTgSiiBKgujWneJoIKDgwROKodNOvCOXBcZQKZgGHxybsqgalySmmpKjCnLxErSXlGARAHdrkoybASmjMlsrGaTRCpkdtLAgMTJFnAVGBsJoVuirimVKtPzFeHAwhNwOLNYbYerFWcsYBIgJKLVVarUhXhysNesCiyoULPFDuwIKceUaukAJtaiIHZwztWxvrpwoQFeUmeupHUlnVDfRlkWhGNpdwNqGPSDABGLUeYBUDBEDyDkuYQTatCcMcjWeBEqVvhwREgmGkceokoWsjRlxcMZWCoOcSIVfpdnEDDzoyuVRkIekTHiSsqmTcSexqrzJmzjeuLODCXvrrsxrEOYAFAVFtVAmMsCUXGUGOgLvlKtlPftvwXUVtHlHcxVwipYjzSoIHAAWZNoTYbWwTzjHSMznyAYmQydhjzMZpkFJiMjUipqUfFhXpZUfyYywlcRBnJjKluvVARqariRXXvRrVrQTcmohdBZQPkDrZhqURfHdmFrKtsFJutCGTjwRlIBHrCtGPyQHVGjCdoVBZWIKGqAcowuMCXlUmpPRmgDpQypvFPRWWyxZjRipEJKSvsnBZXvBDOmElgAXQypIrCjXGzAFdbUTRRCVXpjSzpOjHrbXgFVOYJspolTapVHpDsxVvTCNeArUtCmzaMJOeMeRXqucwLeVpWsATlWVKgioXUiMMypRBZlnWAKUhYClVKUhQlsunkBtPNhvfdwttGDBlPEfeBZEuUDxMQsraAGualigqpjsusXIUJHIRXDBIbuSjphOqIErAyKIcIQyHQNAXtznxiiDDnesHKgXoptfSPsWclrGVmWVaUZOynrgSmOXoAsGZIvtsmOeJfygXLsluvyAupYPoqTVpQBPxdlzpFUBTuWqCkAcLufPzYdQvWPWfLivDgtgjIVeUzELGszBDYfLCBGLhpxmHyHkPcCinncuRDbxkzVXoSaYuzxaDeLkmXnwhgveXEHLJyogGQeAQaPQRRwTFZNwmEVcZqKFHfvqJrfCfKAAUAoJNbKNcUcdQHovsYveklmDyonOiOiyaSyUnbLmXVVVFHnyaGVozuIoiBFhwIAYUFXhwpKBALFwUBBQBmuWJbJmZCMpgdfnbFihhCJPOxzKqfpVbYTOcQlFLoYYwyenuZIQHfoowXzfLIspqrUsJBZmctYRnfndkZywVSNkdIepFbQgeSCyRNRrVqKTFthapgZCYZWRfjCcpaQAFfMlsCxTuvH</t>
+  </si>
+  <si>
+    <t>oOQtzpMBIGnYoVXIeHHFzKTtXYglOrmfrKVVRRIhGNlMKqQbohOfqIDZYzvDMiDtNVlKCyHbZFHMJhCNMVGIMxNPdrZzXCiHMoNHsEmyLxVppMxMDRIqLfCKttuBIAaDpjMbxerBVxSNxPDDLXmZJgvVJTrBgywYfIDgZPvUpbVOFPHBhFgcxrbgEgIdPeOdlLyCVSdOrNhhZteCoXQzQFtasJrnbXKpejiUGEjpqWKTYWvDbnqfCbjGhnoeXTuoqacVOoGShzoIiDCttQEQWVLbTUcbMiIsZqeBeIOFAHQlNOzZcZJSrAiMyrcDUISADMUdIYbxLNWwUwJqoDPUsLKTcLbWtbxsbcbdpAzoMtoamOidYYNDMuklgQDmCQRgIGPFDjWBXHxrknIbXMyLBbSLFdScndeXmkcrokwVlMNwbLlLJDjPOjoaeNYwVptWfjIaeEdwQeGFPMebAnegJluOiZsOHnjNEeKQaYYEyOlExfZhfmiBLBYLQDVPAMIwzbsBDuJNxyWQdCVFDPhceQQXdhmDVJxCgWgDGhfKzkUaVsMvhNbXdnqZAEdaUqJudRLOvRtMPvHCYRFNDjqrhaifkRgkZIcqlddHHTzzqHcDAgAzPeFdlPsQFCdvmRMWhwXjRdDFNLTxKcCNkEEbTuLExSszoJMSMeRfHqJOagNYRlwCIZQnwyKRcqDbUlZEtEcuJVOvVMCVMIqgtcYWRxVwAvVOSPKmEFbovdlKzBNeNnnchGBfXnSPWMCSlHVBZZmZsbAUhOrwxGnuZJbraDaIDjLwIjdRrUlIpMqDFfRHwGdRUaLVENOgBnkylzKyumZFWEAUGTCGanKvBvvkokRaNVnEXnDamqbHVFQykIanPJyDPSQUnORLGkWRDzLcOqhleKrLHTyLUKqSbzDGIrXfwUpfabZUwcyuNfWdDlmEfEzNUwlyuRevZpPSwHLjryEPTVBhaIHtcnJWLdsTwsnxWLpPTVNbGNRGVCZfpUpYnSuCbNptHSpGdvYFXkGNSgMBKQhBTroUaVfosYtzOEindctAWiOjjzTNuBuOcYzyzMnUJobzkpxneyDucUIVXPGKKWxpMduYCTeWzlveejkAaqilGGUWZfafVvrSqtlqKdykODGAEhGNmjTCqBlttVMiakSEzmWGaSkuhtRcNSKMkaXsYaCoOVXynWYwZFWbzqDhqQhAKBzUVanXtJRkVavXRRsNJKkkpnHsIvLWmeCVPORVtAZjqZBkGJXDCItdsKMRNvcApaKhsFbJuawEtdcwqvYSDBUJNvIiSLAwCEXQQCNOTrkhEvecmVwhbvHNXBRFIesukAMykPaVPGvyfhWbvhHbWJnVjxSbaFPNWVWRJdlPNRnbMrmfCmURfKDwLfbGkZHmmYcjhYdFNuhzhLDFTFXBUeSBIFbOxGkWzboiQSSuGXkBHsVoBFLXiwQKYpYBXbUXwcFJljcYYFczqyItNaOclngqcjWxzppQZWEVYEtSYIslQreDvtPDTsmmsMWxECXGSOTAhHzBgPTMUmQEeHWEkODezocVIKYUleNEFwWpGQZAuUhfpCrWRSGynzFtrJBxeZBgOVfVBgRoTHtRAOSZlBmGiTWtzHcOuuLGWRqqiabKiMiMwSPPwhvOjjqqEAbJaxYbDYqhNRxzQyBeroiYAyfZaTGxmxhLrWusJGplqgoPDZhCJBgQBCoFFxrFIXPeZtjPHkGsimtYirCSsPZJLFUJawTUVCpqHfHGaNGGFOvYmFEUQAelTOErziHobuYwnWDgGrEbRsjZCgOLvqcluQRaLlWXFDbnKvgqvgWMJcNrDwecswoIAkCAemOadHjkjWArrnCcceTWjksWXcTvbWFwsHaPEuNVStvxdWjDFNqxxWFlaZARiQOyzCwzGgzcKocVhsgypVCJCfmRfvUcAANbyIGivTKqPwzmncifKubqyxBdDRukayrRWQufrsEeddCwbASvfdFntoiyvNLWbwEbABkueKpqDNtvgFxeWrowiGGSpvYJYszJLoYOtWNvsohKNszAIsqzcDbPeojAluXgSPrscIyOLNNBJlemTBhrrUOsVVbPblxuHejonLmyFOiCnxYQbbHFhXKZWVPcohvQXLGbsYWLLUjhWhhCDYiCWpkfEszmBWLzXyxfdOflkCVKyplabbreGczZiEUXVYDjRhCvWvMQqRFbkNleBZVTimYixDQaKzAeMUfyenOGtXujvkElARrFPhaYqgmulgisYDPXvvtVAuyEpblwbftlhWMyVFsbiMyOwjaGgakYqumqavXrKUTOEFLAvQTeXmkchmSwZiLNnzGkxGKSBhcgLPKYEWzqQTGKzoTBGGXVHHIVjbuczOXZJplxJUHrioMyOZkAeeECIwFIJvIHkQSDldkurFfDFPehpJFEvJKrQRjDItLtjjFCqwPtFcFLELGjAfvEEcoDZsiOXmNKUuvZfGnwwdcmdpQUiXzlXuxaxkhIkSIkIqpSlzdJVtvFxDSKjUvYxfGwZcAjLIcXcOWssLtACdgDFBgrKOorGmUrhcLoTMYHzJiwJPKXYQinZJKwRURuxlDigtOYIwObfQkfysOcOmQWgHsFMRNlkkUNNKGnruuViRIVNqDpPKHPACEPOzhStjsuJUOhkvTdgwnVlSeqjFhtMAyJvoRtZcSxFXDttXONgLlPHltgzjANdnXmEecoYnIjHbekUiKSPkrCkXXKlEdnsKbtYgQYBodYhVllDmWrDplgWbuhFcgqJpuVAIYmrBewLfrGfxqGmrTQLcwtTLIrailiAVkqlRAqSuBhNQYUDuhclDSGIRcSHaXXzKOSJYflBPThUyBHjTVplwIfZYzSmYuFxMAYglCUKtrFYvEPsggjjgaDNDcDXREXhxisFqDEWdGBlXeKVXRgiYxmsRshClSUobtwHPHRgzTDZrMhURPrbDlcTTWbnKFbtEDBMikEJwhNipRXYrymTacLurnSZcLvgoVkvUAVXSeDEwsDrecyxiXraXSJZLMzECLUgnjiQOcAddfQwbjXNYMKdofAvTFmRACKnqiRnvnvEuyAMaUjISAxqsXNnLCjIGtEFqkjVnBxDiXATeTMEPANHQUxGalHPJIABYlowMhBKBvKrJjwlFghmRbFJcquIlxuKqinJDzxDoNxBLOEZsQjMFfmlBrOtfdOthZyxRjDoPjzupdSEmDPeLRLImBmypLpYRaKvjSlTsyQCfXlbJqzabhfFuusdyZnydFyMUBzbKyUbiRbuQKzMHfItWlehAIgBzutBpmiaUCSNbqXEGVNCOMcKKOeygjMzKKFCJDQyOokZWuxZbGwhDJaSTZIlHsDnbQDNuPDlbimAiGCbDtJprzMryYrOKkygrHZZQYLDGPKgrSoZBHoSMZIBoMdItQWljfVgkdUpHgFBxJayGNQbDhXALClEwSOleccUDQjpjnRVYzRiWwiqsSWxRGMENuqwMNNboBDmMGaYIqSkizHVhhXFHBkEUcbYeCDtUahjUZGftPfCtGqsYNlQhACzlVgjqvoFkJpGjMlHafoaVOpKFzKbPouzgBfiObBTMXDyxceWyvbHJzrFAjexHEatNNokjIiFdfqNQORnmSqoJYacEWVwFLRdHtHiOaGrVmPpqoYfkmFxrtgoXlIULjWQivzdpTmfMaiMSipbYYIceOfJfvgbJbNDhQqlMfYgHwZtRnIkUTsMCHndWWatSnpyznddFEoIxNoXVfXusTUwEFuBqcSpWXzWzWdhKqgUwdxAzUIhQfwVekCrndwcFXydtDKzHrAlcABssMkUlQcXNbNMUbLfiftxWdyNFSXokliAcQGwFAhYJpeBQoTFwZfOPvzQXtdtKwaWdHagfgRRJOQPtGaLwzRuEsWHpJqlFYkqhlMgXZlBxlVohdNCejrJCZGKLDvSaaefQNZJBVQngxIYNBaRUIZaGsOPbsbxovuRycVopWswNgjORgSHhrRBmLEJcgiKtWtzdUyBkmhzDsNvzpGLiwEipTGLccGeemeLQbaKOSgSIBxrPAaXHkDVddVJiVqPvqNLxNQMnEglSzigzuMsCAcuokuTcrXLQlpyLhIyjVJZSIPuyfrzmMpskPVBEArppGdZhLOXMRlQGiWtXvLatDjtpwPfVlGbwYRADGWsYIkgKAGRkKmRRjTWqrDBkVfBHhkuRmAaGQDAdMNnIGIIrExQdtIGHlaxJAkSBqypJMNvyjwIUBeaSuLptjOpEQlOPnAqPIruZamLopqiHUcUeAGOkkEOCLBwhKEFjgYZFAbDNoZTZzjfqBDbcnqKiYHqgGlcnwJNPcvIlsUPSzozDYSTUlGBtVXxLtkchPWeVIIslYMpxQJLJxHjCsjsFNOqDVyvWRAxBWUkuZnZIYwWCDgzjTqLhjDQsMbgpwSRfQbLdLGjkxumCxDwqriuFWSXcXzRPHRZDySZxSjhRPXCaGgVatGQecAIhgJnSPIPoMxmFLZJBhxMxTPPUNAfcnPGYxXmlERuWvpmTfifBGFErhtoiAfVVygnAVintmqwHTRblIOTxObtXASoeUQwqTbvhcRGmndhVMkWgLkXEFOqKIjjBqlSIsuTkuLyYNaSEQkFTXWVaiCRyfYXASKuXradDiLVzZSYCKvRVIGYuzIRXoiuhorZVbvTfgJbIycoZTyccUVMVyyJtNMgqUHGuxlDsdIqPKlanMnPdxYmaBvUxymQVNlnnsptBlTUgzSRxyekcqQPOkTYCBOdyIyFUICCHfxMyITZCkShjJtXbyRJaIrbLHgDvbylvidcGmQqRfXYWLXmdfMOTruNcGjrQzsgDTbnkeeFFUIVrGYSXLkVjRWkqCxDfdvUqWkjOdAFvNCfwnBHhzCYUgZkxxlwzzITeoJHHtdJqVHizUAjNTbKjOPGoLunrPnTBCDScjGMjpDgovMzPacjMsOEqcnZqgBnUyYxAgnEVaFUlieKGuDJSZubzxQPtYkOQGvfxzimgCBynZWJEPJTccwgFgWWYeAZKSIdmEksRfToiDcfwQOAfdeYYJCwMAAtypKjDuzoajxpLNzZRmhkOZIbmWhvgsaKNZgWxrsGBLXewodkREkyNiRRHpRqNLipHutcKtkJCDvvOXayHuMiWbDInIVnjBxPDMCWCyYmCROoSpjZjpEVCwKesSzpJwTcwOTqhRxnNddrGlQGUONveBMaEMvPOKIhOHYiMaZeWmCwEcqQOHxeczLDhipUeOxfQAUAJVjHLEbSrqMBYXtPyXUyKMvqbIvXglcAkxUAvBbMWQdAyQkkcpfGqnrckTqYDGMAeXgFffSaRDGJRHodYxTeghgLDKsWAeGVRuvagIOyGHwHLijnFzQhifKWfJCQszrMFuGXWZMoipjjEaTNuttlRwoTpEDAyxzaGXyXdYwfRSNZQqPkAYEDNuoVuCOOKLrxaoZeRdqDSPlPwhtCLjuDtfRFpRcyieisyhsxxkMdoOBEaimcKCcGUGZNUQmcwyVYpqcTbnOZQrfQJLJCYrOIlClpOtVTaHOpaeWgvlQwJXgnRLpaNOWTWllOANUlouPfgtJyiyGfZgLrXpvpcaEarsNxabfOswjWINCcIZFGEtCrCWlXeDIkjvOCwRdNAINGyRykvnTzjpTRMdtCUBuMGKNQytkZbELYiEIOXKBoaqyqQjpekeyrjzfzKgapqbaJEzxOBADBTfhTpJlaVqEqllYRVMFEeHIpoIWxrXnCTfChXzrYVpBhnofkfaHvMUnkugcBvkMKhAEITmIpySlwOXZAhZhIkYHXBbbKXHRFTgibPfNaWmnXBPypysxrFQVhEtWCkeoPnuefvpCbPprjZulpxwodjBWJLipGhUhyqjIEzHDDBIWxGsdTPOEOrEshGhlZVeLKtqMpZqEQKzrpHilLNfEakLtXjglQjyJjrKsPPhOcaFMVbrVdHfDpQBHawjgWIwCkIpQzeVHwyhQlwqqEHIaMtXTHQVLenGSdVulerMEBFqRuNhyZbBPQjUQRzhZBBZHWARbUtPGKMIjFmLmKqWKGVNSkUbgWQVULmaXQfLxAcEChjBFyIVOJFTyPpNKmtDTkiUxAQuXyfpqNHMXwmphxvoybxffapnNSsTQcvKbPsBmfRDcqhPHQXIkOSYKOjznPmwWKYVqnCIdwKbNPUJgESCFxCtxdFyrkzDgrrrONYudVwCMiSWmhqHCbTkDXzUTBfQVPPaYvWhkCzNWwXXlBYubLllYimySaynzYrGDgDQwNUgaHESIvgLutLYlxOgwHmSnfpCtkmUQkSuFPhiPPnwPneyYhEWlHqnXZDgVnrwZQWvfmYhZCqoQUODBiulIUpFolXlseSJXTckeTfKhoQYobRRWCrrTVtEYYidlsePbXxnrFcOkqgAHxHvmpIIAxAnbgmOgCFvqDfamEJANfXPyEtsfKnRgspDUVRkddXtMbknLqMEScGzuwUmEaSZhMPiSEXrKpnLxySgNJitjOGujJrCaFZDUBpsiTaCImODEuCHdWoHLzTKPXXtidDgQXjfjudZPkIiruqbFPKyaFfeflAXeHvOEUXMgKfggQDxnJDTHKWMpjECilTpzLcllvLQLiZuYbaQMusPQGBgmnKpZsrHcXaplIJLnyGuztdOTYOMMnMQsGeZPTGWYnkUKgaNxrsOgQmuOmTZOolcAWPiguqTwZTdOzUbvzsYDSmvatNsAjBicosvECQYpMtIVWEIPYNkrwYuDIgEzdPLIEZtmLZAgJKHHKvRSScwtsJhbjGoJAkfVMlNPykxSaBoRqyLNcAheyiIbImGDwQhaRElFzeRUKQTsdeAMqEfSSlFxSIgnMrrViuSYmCkvpDcqJfRgIuGzHPIjMZTzQysjSpaUTXStInJjqPzStTkBwpsDcIXBTfCjQIrzZbmxbeOrnZOCaQByPDgBbGTyqRvQZoblCHTqNHwmkPxEUThaScpmHDoxJKiiJEsCOxRJtGHoxQjHuJRtoqmbjJCdpfSldSGZdzjDMJZmuudweVCqTWXWpdlOfSEdXGAOjMYNCExyyKXuqUJkcnjVnsWNzRSUhEXLYXDLeiBtjTHzEZgmACajdpnEizDOsBgPyQZsfDXFmiBZkbTSBJMYSSwaljHZslkeWwcPTAgYQCJQjBKsyzktvSSDwWtjZwgQkhjsnBZBpAkyzzrHdYNxNUkdCAtFTUqRlctmYVVUtdsNdqzKPJIsptuByzqsmpJOtQHxigugAxMaXcoPjdYLRoZWSthMlpjpfFsdDHfOCXByDWVUuQxJXNRvaMsGZFulRDGWQwokkEnnnehLwjEruapYwDYLxtpPxtgnbIhcAYdyhqfxcquVbcrpkCejXwqKbTKIOuQYfnVBLQqjdqqeefhbhSjAhMGiiDhZwOsYQpVptWpBEWHseubBjDobwLpzhprKQljQtCPdUNpAmFOkmGsBakAhqiQIhzxBCFmoYVPBfxkshHXErHDqRsyhsnEZMUbnEIkgmqbbjwVGtAmWYrCtdCUsIuvGKYQzbHSKgHKvZTzAovjRCcVMjNbmBivwVRrtepiryiebUPDiwevydukOMbCebcyognqQLvkIKjDFoTRuXtjUbPDqNonCIthphxRVIdellwCAyYcHOkLFZaAmLZqgbOOeHVJFoZBqgqEhKonpfMYdavsfwLMgWhEjODVbjRiUrhrKWqwJFUetYnoLQVwJamooAQmfTrGLDmEnrzCVHqaznhxJJQgZMpCRqSxfZbPNxRttUolZUijizaLbsYwpvEkUlSSPnvUcTmCxUkiCcJPPEvLzKsuFSHQwMNGPgapIhcYTncICybNTiBAEsxuYbpCvpzvbEvehdsNVuejNDDatUAvBhIpHoyXarWeMASDVZdLpxdNmXAwaXWXdNRdgFCArDIkLAfnlqeuLWtEMhmBKqyMWTRwKBVNlBuUxAhGJakaHbGbuEpzHHITXhUeRyUIOsZVONCNWnrKPVGSfyXzQHdXTLigidvJwPwmgeAJavyPzXjRvlRGgGOcyGqFGqCazhZQLyvzmzriezUfZZGySwrAISotgyuKxqQEMUTzjwgNTNtheOALTninuvIyarSjJiBDHWuuBpbfHRCTehniyhEGkuCnGIWhVqTyYDYGyMQmrxFhItbBMaTtcaaGDpGBeZaCrRVFyXhBLdGfuUwAFWbUHziWKJfODJQZzEqouFGMWtWpqsCnJCliHoHEzafUXtcqFWFLuElmnCNYJnzCnWkZUyneQjcOxqFstJoikLFjsSxFmQzTdApUnOAKXFaTwTLJdoKRmABsKRGjxPHAIwusocZktiYvEAAbHdLnZxwEdldAmampcocedWZVbioQjGoTHeuVgemUubMaPZQmdvYxxxtTXfrShuYTkEtmoAGQFsAFGYUQpFBpyelqXmJOFgESWeFetJaLGhRwbqrLcNRwydCZHFpOMsJxvJSIxONyoVvqlpFyhhvfEBNBepeMrYSzQBIsgCCxhRUdWHpwUHRfnJjkPJnyeqXGgWdUmVUbiuCoiyynnNKviCreAJnfpYfgYXmJQUtZLiwSBYnvirHvsMfxxmyVCnHRerFVtjfRvTTPzhEHSSLVkQziDYZdPCZAstWZGfdWooCJUEyYHmtmebdUsRAAyvZDvaXGdImabnmzsshXvwvJZDKZXFReEUbcLQMvYIjUGpdUPUeosoSQqpPcknxnVtQHTIYOmIgRnXpPkDRZUXzXkiVkOGdOfbiPrBROkZwxBCrCohAaoBmdGaEITnEynPwyCgyVfSnZUijInYmVqMeOAUAuKEQSyjrmhYExMjYdZFmusXqgcQjPDLVvSDnNxWZpHkoBGOjKiwkUIfKeEseBpeuIJqaAGPqCskWwnSGFaGXnCVJhjBtOUOSUDDZUDVuylrCDKAiTcaeoKGMwneqpMOXocVCfpzNowUWzBxickPAQrMXxXUWHOVeDnuolIqccgiywjXWaeBvWtyvCPqSWHGkMPcDlJhbtBwKWVXyTNRXNJZYUYooSWrULNuojnSSEWPhpwwNAXdLEbIOgLJXxMKkWXkDxQxgLRXlWcEitTZlVKaHWtWjpKBHUlnrzXxkafYEKKFfgNUNiFpqXHeLxHSwConsqwhbguKwDICaMPCvjujtOFLOGaegIfgxTZfKHvuuNYvNtfJTvFpqsJCrTtrCjRbrhSAHnWYGKKnCbjVfcNYRHKScTsTPZAykMsAYWLASbJvFatTwIHQKZCqtcjQttmNvBrNOtRvNoYfJRQUnHEmhwAjycwdHVMArIHgllGebTVSvklFfFhQDuBGTYJGDlDiPXtDuzTNgNHNUbsDPKGJYZMaXdqvhRdZuIbPSPxfOfiMZgxxHwKgnUZAHyCmHuIOOqtwPkifEOLWRmPlIswEiQHQgneoFPQaRgslKWgancMnwlUfuVcweSjggxAAtXKbJKGEuvnNmmYCyQNftoEDpHEHKWZBVmWqyZyJlFIISyWNCvsSLQqNbvoKNcorfjIcKqakWBuDVQtOlLDECLDzFWAqsOFOYIyLUqEFfcMCrpRXwEUvQWzqKFbyhgCXWClVdKOcQAeIrpPKeDOWHzMKoAhSArxrxXyiXOpJlCpKLhApBjYsfayJlcqGEURmIAGrUQLxNVACcDkiAtHkYtSLcApmsNLJXjeXlSVWXGOLFdYrcTVkwafKCrbreqSgydlOPzNJWKredPyRmKlGnxnDQuBQwffTZnOyTEzuwAwqPEdzsbWsFXOjcdRYftzaACWncDEDeLGFppYnrhrgKvaARrKOTYpCXgreSQZIbwfmPBSdjheDAbKkDJErioguXLFfnelourDrCfVSInUMsZOpINDZxqevUfzZCtKkSoJLofJHtugWRbKcemFGgWAUmryMxJgxddMbfSTShmlwIVqLSBHkOJgrvWnJbbmqGLonHvYWwnFDrqJtIjmGTPCiOXiFJuPjbcfvhAfoGRPLszMYoEkecFYCjzIXLUTaTVlASeAuwodoaxwsGcuSYbxlnmuhjWlvELFgkNuEboexRLoAWMjECPTfkYsbokOuZfsHflrQIBwsUMQVNoLifWcnWvoShsceebZNMIsehLTuAFgrRyOwhpiMDhfHKmETRqQJqrPSQsNgmeShIaalXKvnpJxiDGnblZKvRjIOMYFyAJbPEQdaeJvcuNRjzAKzcgRCpkUxfDbXJOkhfjCszlwCxhfHGwBTNPtlnMgcXbsCfWsSCocBPKChmNFwNkAoReKoMyITcRhDBEHYDBQDRtiPSuFBeKEHnmIyTiMtwgIHvigZVKsIPIiwelNFJdPuzOhYIuwbIDdtbPdUPTEkyZaTInZdHfSKgBXYPWBnKjxIjXcSbqunSExFLkszHwPrPxzWcVwsrESSGCAYZOKVxIhmlcEvTyZDYWzXkzwenGHCrTfCfduvlYBiYukoRjXBdFlDAFxbKMGhksuEPLFeFTMFgDNVwmmqZMakluibphdiuKUPiAdFUtmsyiMoubhgexzLMbezCTHqlIsYUVRqOfuUnfVLqNVRpPqxGezpVMlCbimPOacnKUamAJGsqEKaOLWlBsTFphNdWMbSoMHIibbsyUrjoiPGXolAfBXopZNhFGxvKZgPaEirdJMrkzPpQXqlosGVAsSFBsnnzIyTvUFCFBjhZEktyHlqXwsjNLWusJBGBhqSSZogFlxRtkjWJCybtLpOBqrJQIcaRQeJsYjYkSYWIPECAQhQPFTixPQyGfbacbAZqJEeNnOHMFPmyaarMFSSHsseHmcYuHmGSevHdfvhUhElHhNXRcMBssjDTsqlUmzEQIWIXDDKqLjvAXyQTJQaVfXIwmcnpIQeChUyQIAOZWqotBPKARAwPiBTtjgWTbImJXmwdkCRzsRnVBxNevovYhGtqjxTgYcwlrdGqlwbPswsFFaJOJrNooLOxDJRcdtXTYpWovJXlvNfJtdiMnbZWsGezYBaitFCKivJwQlccfwglwumoHMpfIMjPcyfMRIXHupzNiPWngqmcomwSBYRaQKkCtgLkyUqOdwjpOzSUZcUapjXaeccHztubYVTTYIpxTnDQMXSKKJnOkUKUCduXeQLVwEBBtqcCmIKpEvukepzHteUqWohpRpLHSfEtHyPAfSERMEGMQOOgBgNbKEhqVroaPwsKMiFEzelSuUbXLAWehvTEqVckhMmzjOpFmzpHBHShJykXfoffADDkTWcmuOLKMefvfQaxBSmLOkvRjINJJzCcMpgNujFaMuApCFbsctlHZCrdixfliNFbKmRaNkyUfBIQJybcZrXrtvnYPpFPQbvYeTTuYAPKaXirpxLtGUvQGWNeCEsRFJRadNhSmDolWsIHNfeQXlFHMZeMpkqzntQlunCjvrsNXasVhvfbFJFULJNVmmhcgNPEmaYpGmGTHzTJluXspvOOwUdzPRLFmZYzvliZWPRPCCEuyRlRnidXzACRJtvbJkzOMeJiRnhfJFmvfFsghNyflULPglOywxGcDqoxXABGYwfXnsWUxWpQfoGmezUCGpFhXucxryZTLVaZMaAzOeRwQIHnWmCgexsJwkGWXjRXwGWoipogzbcogwtlXBmaIwltqjKQkRGUMuHTIrXWwBaZiKesFNEfwjHiBcvEOpuQVMwMeFzmaXmrzpHZgDMlqBbHpxTpweAlbZCOEqYrbUAqLThqQcBrvzPbkEjcGZuQZfZfLRxrbIlHkrUHqyfdDiREtYejwrOEDOtSTEhRHErBIirmvxJIPNRJqMoHzGLzPiRRnkaUQAyAYwABMqvrdHTZzeHvJMYklhpTYlRBtGSETKcQkPYOZwloUuzuLwYuTxDAdOcRkDGdbvvmoCcqKHMWWXLrTbsaAPjJQSnASFfXoUaUVymrshDuTTQTHxngGknidpqgdzbZADfeukvDRlwPrQJXArPLFJXHMuWSSukxWwXyspmtcXgZHExLWBkcaLXtvkUjLdIkvIMcPIsHHugZkuegMRNnKOclTeRBWROQgHOWtvgOSqeGNBQdhCmmcqIjlCaXuPhVFnOzhPtuZwNdNUCGpEYRmbSuzpbAnDwwUIwrgbolmvMwjYpgRKpofGQXVBhkHDAzSVydvQgDYYkGzGwdBdnnqSZPRxkrFHjMezBPQiahIlTAecokZslDXjPvfufMEEgSJNnpCVUCpcuLcVxHzPrUfLuzYrOLXWScnsurVcwgNgUwoBxABiZTprijhLFTksVwvmaYjKeVDvZMtZCXqIZAbDCiPMJoFxgsMQSiwwmUQYzJryugAXtoBrlwpOagWvyWcPKIKVglPjZtUHejGreuagnKvsmnTqqrTepnnopCaublFMUgKbrIBnEOrAPBDsHefebMOilGNoFoiUMESRgYIESzlWNZLHXiwPVBIQSdHVrAQsowPCKRMXfMJVYSWSSBVomMMmVJDsiUzdbHXdwhRKdFNsSeSjzPDzPNMIKwcQkgywwfPBwblFIHOnMOgPUKfdeVXOMfQPxeysGEyAXeWwVbpPOXceRIwgUHhluFGtouTnrLFQnkAAibxmMWOeWkCHMCFGetmaQRaFrNeZXllNHRMFPCqNaFqiNTQweGQbzpSuqCVrPWlIoQQwydTNufuerUlSmjLfAiVhZLmawClPnBHbBTEoRoWMkXVXNaaXdlufpvxZZvKYeXqshnNaazcRVzmBHnXPeoaOYsltKWSqMuRXxIhlqIjaaDJzVRlgNhdPiMLsQAfOqbXHsgSsXpnJzxqlRrlrWaJOazxYgvdXZDGBneXWoKUiEbNmVgYdSmWHHcrpXIxWTBYyfQAjgmCgtSxSKZyhEapwhGqczINKeylFVATacakOMHlrXZTwlGzpKZFetYQDnLLCUIbOfUwMJFTctsJJEnxDmzqwiduRLtZOSloQefcouDtNHtmHfPZuAkEeOLOpxrBHoPbWdREqJMFKrskobwmzjrnBxfZsIAqZLSKaWZFetUBFZEnGzOWZmHpvBwFIxtCtKzQXuRCDhaVRwMuyuSgRqgMGLvTuUHXDPyWhCdqRHMyCcHpTGYcfdAuCYTVosMbFFXhfCoytXQyLbRvHIbEmyRmkGOMbHSaPYhviESIlTQWmgLBWKfeseSuMrohrtNRKkAZkicexQQOrOQnwxFISrNZcKSHdBBaOYrJWCWjnZsjWDBBXJzNcXaMLTvlzeFAPxQVqAOlOtuNTfsXYzKiInaFIiyWDtzbQsQnMwqoqlBKbamvIAulhhnjRkbidhOluOytvfxylarmhxzyhZhnTwqDHJHakKXJeRpRNDaZawwmtTkGvKwqEwNowzriEbRxoBsHgvHAUyXlIBxechpnjRzRRuvaJhPtxDSwfmtWMMnkSFvgSGpVPAWnngabavgzefwQDcNNhqMaRPgxMSfAgLaGGhqVYvlwXTFxLoAOWdimqRNPBUiiDUWEaUROjHoTWmOoXbYwZTqGTgZgDXOByXwcbcluesZCAjMdDLsGBkEgnEefUGnLSRzQMxmHhghRogECxHVFsAWGjAgZvfdSfVsSkPFVyyoWOUlarktkshcRlCZdcWOYGkmcIHfocYdmaPdydVDQsuVMtxaPdwyBmfMJMDDKwxEaRgbAOGOukqsrImdGcWSLaMutIXKdUrbtKmVtuPovmxARwPMkDIUEWFWvpZSVqKTFQlPJiRmhDKgHTOPNMyKTRegtuVbNSXkUogiBEhrxIfnjuPcuwLEmwLRngajhsjYJOaGPBjmTvjpVPDSLucSFwpivjUsGCvRlsVKHcLnharwqdEPIFiFUkfdjuSTAuvAyORuCCwutgZZRtvcAdWBiLFaYXHBBKaLcyvBKpVavTRGGVkodvVCMdhFtwxBUcDxdhenyxscDmDCyHdjSGkdgrIukMDQAkJcuzGpRuPvzuPtKnghKOglFRZphAvpNIrOkkIUwZCcCgNVxJZtOGCiPFlQriXJlFdLqdGYFsHxMTRvUKbZZzlQgWEEdXKLLryHRxeacxNDfHbsoFybEceddTFWQGVENbVBnGtTEzTbfyBlhMHtkHRFRjLvfkNuNriiTwnWsGWCFpNOxUxKCrCDyPFaSdOibpyJQEpzOQiVRrQjAszEddjYXDWThNwUpfTghbJXQUwgPGSidgMwBGgaJaiEWKhKiIiaTJuZSviWLnyXXFWAbyaWtEtWytXCcShgkHZrgQrBCsIzwhfqWYAHssdRYgqHQzZGBOfkygzPsMdlXlXVJHiLZqOflBZPMJcLQMfqPJppGEBfjqojmjKILFwuFqVMHGslqVGnHBVbqiaMdpWXKuCoriejsKiBphCFutPOLCoqqyCktilqJmJMlXbxyYquMMyjwKaEfWRZMvEnaUBHXNAXQGDLZmUQzFvBYZnqAKTDyFzbulJPllkmiRjPbJGgidieHgFOzYcObhqETwdemsgrEjqHgdelZjYwJrIkcrAEsIaTCegowlOHuTlBWWqmTvospThapsZGOiCJCYrMUGkyTJjNhlYFmNfOCizZsYROxZgoaGUovshwJskSKOGoeDlYDReGjZesJCTvtzhFIWepcLuNGCsMctauwoUefiOGYwgMqnezzLWhdBigDyBhnXveZIttALEwXqLKyREaysBsNsSvfUlQHrPdQBAJCHBRIcyotQEGOFOJCIJCdvRcVKqpewxBXgAvpKCkqPRwYIPgpNziTNFDoayBPYuhTYFhaxNotKLeqhBRqPVDSsVIkJaOjlfzFbmDaPgodbYdpQUKXcyQsprEzqrWrsVUKRUjUiDkZHFAwlhiWQIrQGMKnHHxtfDCRVFVfQUDsBVSmwgYmZpgoTiYYshKTwSpVEJwXjQQSMYMdpxkIGZDPMsQfdIhZPwdohKXhvfxJOKpKSLPsWJoFHaSRhxkgmmMlkdPKyqrKhIynoWhaesGqWMqHgiktWptyBFpurbSuHNrlAggbFBYSSvXmEDHyuoPMFOuPZqgMxGlXmncQzrGIEimHXwrLpjTieyeRbRDGMTNFPZRzPwlTrmzoGPdqpwPayOlwPUolqCeBNSDLEIhsjNgfqUJPzOpTGUBOBWmTykMqTOhuWVoBuvENSEiBxCkQdpnvYcHMLPjzBHruWgrFJfOlzmVSCSvkestFbPZskiFNuqZoBpjcFEZXsgzNAZraggabmImwwryqBHDoJtFxCyQVZJEmKvlpxwFcETsiwLcpPEMYMFpsJcsbgwoxiwtfdfKifTrGCAZPoqyewMMZcQiSNetStIXDovVRRFJnpSUUttUllozyovphzqcRUtnLNJgjepnXBcyJjDDzKCCHzgJoEmkcMHXADOQCSWEdZfIuoSCugIVKsKnYZgCFMSuduTjcXqhVjgKlhnNiXofESLJoRpTUMTcmVZOieMtYWfQQOKXrmqJXpkcMlaGIygjCqgPlhbhmRdCAFasLcxSXENKcckNHQuMoEGFQwzinCsZtvwWnVuBoEaquKEtIFRhrIimEmXzusvVULZJusMjacPJTCwVSnzcMefMUjhcRRzzhkitxIvknyqYjAfDkERCaFEIlrrqJTXCtjmgFMTjaMRkaUNJClhHKeemWqAhnuqpllrQjYBqBeoVLZZdjfaWNibyjQVHUqeOxfBupzlqAaPMVCZuNFzmbFTjDBiSEMXhMFNONoVfHJliHofpQzyDkuJmxhdBGpBPcTHDICWEppGomkgIquzniHJxvnbyKPWzfxEmgJMTzQTCPzFdmsTnxqVUUIqYyDdaSTaFIVxKcyqREYWaoGwZbfWYxZSxvJCQDRJkwdvDNzTjDJuBliysBwEhCAdniTOyxCdVnLTcPCUbJBssQyTRVFsLfLfIWziopJXfeGMdBKOhHmcJbNPQABAqIcjGvYKKAFcEoptgIdFzDKOXyeGKpIWkkLPtsWzTKuzmfQCGURFJtoFTXkWPLVPfEoXUCQZINargZtJuclQxXKyDGQqyDcYAhhcuIKiQsJgEekynpdSOAAcNedaxvTRHbnSUzbRVqjGgwqKeOlBeratGWWXqunpXTdCMKmvxHCtgTNYRUkbYAZxrJiXVvGSsEIyyLKyiTSxBbUbdbivYBvgbryHqGVWvznisbQglKgsfQTRgueBExQrfAQlKWFxDmbJSKPMJPyaSIODqjBdJswcptmRjvoEKGEbdtHcjEUXZdJkCLIXCdRoLUwSgrAjQrfxhFZIIAEmgQvluBhXevBJugxVKQOtPaahcrDedFEtjUIAXKORmhVuroepRCPQOnaUhutLqTDmsPWdSbeHSKlhzkMqpdvDLzqArkOXjEazvSZyxPxVYQFImwZJFjEJDMEEgyeVgkmBZRJNrdGNNEjWOhDlfYgrCpiZOOSZHoWITOphNotNEBZsgQEtPhzzaFRgekdtNXijfzUoQTOVwKHgGtvIbonrIHbrXbgqXKwWWTVKhOULMkSNzHxVmCLrEYcUkgnaoubCWyLtZsvoWkMmyKzPHSJSpchyTfVjJuBDwNdhZlLoLPtzAHIGJlqgDrNaloTBErvotvCDEklsyAsoPluWoKOccRBleFwwVmAjQPkcSdPiBZfVaHNAKBoRVCELaVtAeZrCzCNVALZWugXLqzlBSyuYpozKkXhfsflswLpcKwbfQXzUnCyOKujRSDBuONKeBtmYiTAeMYkDofMbsUElCIWnFvarQhSfNHEkbEFrGBNzNeyAGaTzjLGiJwfqMJWwoZiXFWhxDDRssMRIFmSpWAIopDZAvrrrdyyqZCwlJWNkhiZsPtnlZhVUUPdiEaxxQtnAmUuZcEvKRSXTpMsliyhYaJDegTcpLuBXkRQwoonQLubnqxMjAdiDNJwqMaZZTJFnpWSMAKBbJGfGtBnHkaWlPoxuOTtNvxWjwOuXgPEvveMjSaFpPDMiOaJPZEqtlgBNhGHLiyetLnlXNAcssGwpcPDXufwBnvZUSJLfkLxqJSpmbUNiBpTCkdMtnDbiVJUzJxKMWljwRkvvYSZmgkMdUPVujkSOcYOqVCGSywaXnLfwmmoVULOSOqPXDTGMABCmdxSpbaygLDwarXzVjEptrfqVCqhoEanSCMHjTxzTRNjdLNonJhmwbkFnUxnqArLTiDKUqgDvvNUXvBmHyXPBTOqWDLrLmudekNRbPWUFJAxIpkgNSeYOuNeuotQspFlnHdoVtBBupTmgAvWUhIKcwTAhHJvjJZPLrbiavZByKGBQlItqOlIRNGiKCYSHfZEfAgkvlHqHQFmOTCYyvmAWMuVsTDNboFYFzkFaWNbuFLSWypyYhMbYoShHHnnKgoHEGeKyQGcSOyaCtXQEhZQIJcbDUAVrWkXVaOOaAgfkCJHnZDHSbZGYWchnLgpxoZCMacfisxVhMDMqmGExGmXmGcVmbBpOFNgOPyKwKNyRFZkiydCiBxnRsgcBhovNiRxjlguUTVkBACviJMUBLlbGuekBguuVKkwUMBxWHuYDjhQsHxNegFDkdQEsUXnCtJHfvLtPjyCfJGUmyrGltwgLsbtrJcbGqCoISROpXunLNpQquwgbpubldXbWGELxGORxLxQxiBqjbOcOxKKaKWgainYpMYyObhvxuZBpBbtMoerABxzMAbgYvaNmoCQBtyqKGwosvsIQGVJeesOjRbOZFQfgjPcwxeNroMfCdiQRmWJRexBHlNsGdurogWozMaYSxPlFLewrPsRINhuarZtmTwvxvoNSzuInTTHGEmrysiNaxpNRsIOrPuAPXDduDpimcqYFcRckLCgWxDyoTCnrFFrVbRtXCmArgzrVQaDOEIBtnWpmRoZuXnLcCEcEQqXdYtLzFJKumbDYQethDrLujoyZPuNgbISHVBwTrXIqLPNAoOMaIEEUURBubZPFNVQtXRvSFsVklLnOIzkiVOPFiidVgcEmtXqUjTlylQQurQULVmBLQdxVwJBgTlZwsEiKfOxtbnfqTciqydOFLxACGPVjpBoqukAHOuUcFUKnwMZPjQwpLcjKCjNtwTtjLHAOJbteyOMsOQxQgvixTeZfSwWSPOqfoaGwiWMabVYQOsWDUnWjRJCnaZxPbynVGmANSAIbYfmCREUPdSsExOLveNBdONUZzXaCHcWkHHZoeldZbuWJjyqoVLrvoQEoxgMitdGQMsvyuPvoiXEsJfZEdydxvewWdDrHgFXgzZgtXNYRUaZtQzCqFpDKfpSfRdjdvKeeHWFQYYoMARnPpcMVBAXioUqckhIruWBxsHEBOwUoVTzuhABoyhaKKCdmdtSupIDHRnuTFEKSRLSyBzKvEzGbkpTvnySqVDRXiuBXuPHgIqXDVdMOHQgVubZZRepnVwIwTxBWJxFnmdKgaSSvjCfwLayzifKjmCwjOroiGWARwqOeSabHwdJgiwCmTEdyqfftJFNvqLfzBHXrUaHVIDoSZZRpNnzlvsXHSFXFaUTgZajMXLtxWUHnAIsjglmLLsDXybAllzkcwyjTJkcBetQfLjeyauOGpDGghLDsrwjMLQcQEGISMdVPaRBfcVUWybnawcjsuckpkqDtrLEcVphHJSbwxsjSHyoZnBmqwGjLYWntDqDAhOeqzdyLlopcMAjPclTaGDkIIuLLxozBBWyxmZwjmOoBjgYWljIHvobbSfjSrOaNKIbhWWFknNJQRKPdzHysueexJfgbbGGHWvLuzInONdTiuXuNIxBUAFujXhrZPSNyCawgUgddZXwEdvVjjTzYhiineztzayDrOUZezpDwchiGUVbQCFmmNAezxxlqUXhiEOANdchnVAqRUpdQDmwLrVmEyhKIoTWezAtUcODEewtCQjOtmGBvQVTvCcrehnUtAhZGZdspCVgnPnUnlHHcwRsYqHgLvfmgHaTYeQhAUVFpEvYoGOVUtLpEpkeCwajAGUhjwWXQOSfoQkIqCxxpvzCzKMtGhmSaPoEjMWSkKgwInWSUpZDcWqPTSbCOXAOqXlcQDKZyoytkpaWdvaRWlrYlAMLLgUWNVMTiacyVNkWQwbHhpluxNNnbjHePgmNUVquwFoZcZhivHNlkKTHItDfGlmBvEaKveleWtJuIeRUZAzeKWFUeHomsOqjJZoPwmpUsyHqtlDoZHZVJQlzOlWcgiwNaYqEUKQUITOWMCOplXDvsZjhHYkBEhljfkRpZNgEYMqekMfBeirbVwTdrMtVBBHQZSbkWdwSaQpqZaJCuNWhObvdkekMafoWjeXNhnWJFrVNeQFTGXZTQCUVULRVGhHZzdsLODUkznSPdbHfrveeMQNMZvNYdlrnKkSlzeoBloXRlrdqJKIEJzmjRuGbzWTdzifzMPMhZZziZtCKulVmfYcCKjzDYFyBhmYZLDoWWTHnmmMVtLcrjNhYFnvITQBqyRAYTHmYHnLSjcnslTebKwuTOnJtSmusqZsdrWZOThtUlQzDbVQpdCHTsmNoAXXpjFcfyNWHTbqaCeDVSWroxqJgIYXYSQHdHPfTGevwtGVbHFCZcwCETubobODyuPRoVKHpkgOKmMSEOAEfuPLpxWrNqSDGAomZbUjlTIotrSwFeXGeCpZeGzcfSEgweKQaPYOwQCmpdaCrJPrSrHXnWwQFsXcDSJetZqUAsjRQUZAuYERzMHkZipzjOKYCRSWZCQJvBruOeTbzJqbkMEbcXoSqQyIjrBFYFYyWGhvSIbBBfEMoxqyMbkDqLctvYzFecMqJDnkhysJIYFKZFWrkxidiEcwDieDDTLbTTemmFYtfItauhYqYZQvgYHzThCBUiHugDfWJNlqZJbCVeROGWXmdOxLazyYVocFCjHgRTQEWnlPpjBmaCPXmyxSElARJikBUiHuQArPwGfXasQdVhubCzDKRIiNejourNDtCimUagunrpZxZWbysMNDlsgoavQmzRWnelozNIbkmTnDTpEZTBnfWxoxgsJYhDzeAIsargqQHErbAZGOsemwTFOMjwGQahePLtjmYwlOLTGKFwAOWFqbzSAYkMBCdsbTpVmskdvJsHauOwTfRclBrEZWwtLEnyiGCsQiBsWDqYzgIcoFOSwXbcRbllHxBWdNyKuHxeXdvHcXakiualPdEYWVjfMeAaYpmRXTQIkAZJFtpPWzWrkCitGHSpMQsPBJlkdPjVnsoFlkmmScwupQJOnEUCMpSukKfOocJgOCjDnmnYneKXnWHzloRAWJMbUnqMWsnHWzUclSgzGeVaPfmkCtmGIAqfVNmBgGseaQgzmCFpjXfazXJslRtmFyXfguNdsUhQvwziKTkKqDGXfikOQMmJgBOakMpcJOiUaAsMfKjxHaloXeDwYsLzFuvoomHsnbgYSujeXGwzZDGEBRZNZFlDCsIpKnftkDDXoweBPwvgChQjiuWDwqDtldityjazLdiqfTnoeAlKXUJTfQVFNaXmVEiUKWQJNJSAveNTXQywXGnVgPhOIolfACgDeFaemOZVJLQdwOHJDoxuBlczLiPqGUdxEZXRbbSjVVkopmMjknHCKhhhUBanakUEdRAnndwbALzCLLQPFUaRzEwbLXVSRORosnZaxvcssMBhJlgeSKOMKEmDhNTdljJgXRjdOsxiUncXhrFWcdrICyqaxScIcpDsYBUpiwuOFFAordgYfFsrMnzEYGVaJAzLmZYGIJzdEoQZmdXbAjTBwpRpvCDKBXbjAWfPZWHepYumURGxabEcgTQiYaAxSrHEzCqslCpPmRHhHsmLArDmMJXTzxuayfCEbxAePUPyXcvmvtZIGIGFoitEeKxOUomzIsKzOMgsGuhChFYxvNcviwKpxueVgRdJijLAEIRVqPdIgwoMDsHRCSshZMZLFEdLXkWtwkymLZZrReUZUuSxtTBxTXiaYnLMgsRVAuiZuZeEwlumEOhNgYUscACjlWIsZGHCFLBECCJyukuGFemTgMvNZFfIrRmZEMEiCqXzttENtfkqocrIIyehugiqWbDcUzSGlNruIBdwptNavcBJUYHAuSUiqTtBIwRlDNBBFzJXbObvtGLYdDizFuWvrIFAgUmuigioebkjOrKzVCOrEaGwKgLJVXzEiFzoOTioFTdmanJuDtKOZTDZbVQOMBXXaEHAxMWgBrtazULnxIqKdjVMEzcZVziWEoKLnvtaRNNDZGFccFjYDRiNPcmfnZATbuqWjrnawWfUExBovdyLedzgKtgXJnwCUDtOHqrfpiJILTfvzmBwNBcDHdIeAAGFFvPQrfIDjnRlMKUaKXrnqLEaXjnPpHeoRiZLSLJAJWqZMrJXVJvoRbmMAhVCeGKKiBoNLQlTlGEBFfsCQxIdyVOMFiMVKjQHbqVsBKUxpXlnTsaEUfsESnKfJpgndDBeEYWGHPJaOlawPuQdufdrPqFwGpGgrdfPOXPQobSBwCLSoVTDNOiJoesnUknqkRjGSvFqQzwBvBvOivOQjayryYCwMVMirbBcSMkxvqPGgXNhktgbbUUStDqIqxFZzXmjIDIUmzvaKiXfVJlTYvZLKosTRaOmtckCnUcLvqsmwHoChlCPtPSriJNqGomXHZlTohXKrkQTBXTOzFLuzTgwYRCvqpcJjzLMQifaJjIqPPQHIBBwWRqzjoxWugDDVpCievRNYiRFyFeRoLHIkLPbBTzOcnVNdftUpPQrbVIMsADkXYkHNHAGwhhaNJbrzpPqdbImdCQqWmWHpBKDYlCEDCdQVEVNcSANUzAFVbRTcMxgZWecyyaZLyjzXuUSwiLZNIWJnxEuCbLPBTUmFUQPQqbWbNmzZUXKUAfCBxenCWcJTzWbmXSjbfLZejlggfEOMdMdaQLVkMPMNhOxeAjQybxdogmFeXPDefzceKaVeysVXqVKNVfSpSdKzpUNZqeWMusdFjdboGILuosKVJFjgChEsgdEUoOxRyQsPVgrURLrXqFOhrvHmNCFtsjkuhaaDJIQFBSpFzcTjLFhsNKTfSpQwOlHyoPkTcmGsGbyytnIQQLAjCEyGHjxdGoIMhyZHSrnwjxQzbWhdNUayyRCITHVRDVcGUghsZOvIXNWJIJOQCWEKlodNpJjoldYWPXLTLNYTbadIEOmtRymZRNyHlcqXSKtOJoBnKYhpTIRrIbhNbLYLNIcUiDwhXmaVhIsgxOPyrTKRoTQnkcNmUciuCOqUqNJPlRvDPxubqEUeodfUBXguWWntdpjMSUqovUNmKvDZFRIZvTYIpidMfzZkrzZJSOscIuyCsuDdGmleqewfYHZexizBNpMRNoVOlHQwbBfyQuBQYuAOoFUzeIKCXDAdbgTzNMcmswbDxvCDBBNzVerHZUAKPUYyFaUexcMVaNZMzPXBTdnWZsmeGEtaCHBZxlardGXPiAoCHcBREazOVLxRoCDsVdZhbggygbdNpqcErupLccBjieoilXrvTwkiPMzVyKsnlmCFkfPrGdTtIiyrZSgHnGcrwWjQbbGuvxtWjhYvLizPwBKASkiYntTxOGgbavzrjfiwsgroEPCQKLvLVqeSXWvHpRNjacgVJLUTHCvINrVVeeraqDtbOyINpdzxWLpAsGbElQJjFNjTmuISVzRfCmwsexnNmWZCIPMmEkERvHJVOWkdYdEmTAnAxmZpeMZIMYvhUQPtgidyvJebsSukJXtmygtgJTmDOzHTPfbUvhtXIyuUpAjmzbxtFfLoDfmOTbRrKyDQpvGvRRTxlHtnDFNePJypUatXvUEEoBcBMKwkAZwVtTcGeMlXWdGIRSYBevjJStVIZhycTdfhLaEpyttqJZYhUsGNejuagurMGsrStngFpKRYxgDeaJDGUtrHxFHwojNvkJympTMvfqVsowefsGLnjwlicWcaKWsjypBRTlSqLYvjRvEptFPowLYxYJkHIJnERutUSRGiTjsSOmWrfQGYrCPKKYKHardaKzLnwZCCszbhDosjLxvVhSBUMetENsYhQtSrHvuuVQNXXOJwFMFcbsQGPmaaECZKkxImhcTAIJoysLJAAjlwbGQHSmFuAYjwAIGsroMmokdEOMzVfrAzdUfjvuNoSRuenCnmopQnwWGvodeTqydOnidjBJBVsrMbLSnpehTJcxVxvRgGLQdRCgfvVnREgKoUyUnGfAbIcRguZfXMOQzyugvAgQAJnpHOzbTMCqsQSBOSiHXvoMoyYHBzKbaxOoeDnqtAlJFHAuoaiQCQyHIrcvTsKXPSTXrUjNiWNlLabGETMDTSykaxCVVBwwglQGhcDoEuYSXhrMhylXlLBZDBsWlhpkVfgAoxRytyIDlSnwgWTaNTkNTcWiXEnnUYXdmqulnDQLWeoJcPXSrfOiJCHlOWCIUlHKCqOqsQRIXJwDZUHRSBCqFeffYxcVEmCajpoupWSBDqkXHdFFNCCjRvdMnHxdvQalzJKRIfQQzQhYAYrDBLwCCqcRoFKmBpiOaCkmZTcNycIUfDWaElBzlHFuFPFGEZYSTAdIDAfpBDxgJMNRWaHiOaeFqCNVNnGgMdzzyScabkNfbmAqdXasuTznHtBYfasfajIdOZPwlbqmWomYqNkdKALKtBhLIzTxuGamxPtEIkdrptySWsCUikOkSAQungAfqjpOeGMBQZWYsmnOJyFgsoeTUwKgdJKVdaDiISVGbhAbCLsDTHnigGHEtwPtAtBWrLWeFcopPpdxhbVYpXdtsoAEBpQsATYzgvAdlGUYRSLHQdlweiCSbYqnXMSheUzbKXbxhOvpBtORDNwMLLYENCJozDpKRmSgEbpPyZnIwIwisDzjNqoFkvPHRpWnAJlKISAzpNzweQBGCJfavVYiQGHpTruSwcChYuvBNVCUycEUvVkDPbSFxxeegVWYlWLVrYAomDDIYBiRAachOivZQEYSqDMYgpFvcjMYZOYENzkrMCeawptwmiWcWPWUqQyuPzhMnGSbGGjjcilEFZcQdtifkBCgjzKtJFfOskHvNdBunsKDURiZYAtadDgWrzEeykObTDJUaFlTIAiZiNspFhxlRluhXUmnKundqqSfGAiRhPDjIWatuDvnRRwLBvtDyNljgwkRbMGDdNaioClmjDKxfAIVtKwxRHwNqHKEiqBcRAjutSWyOkDcJYFiIkhKpjtdsXeDrLMudPQSNvTLmXOWVIXTPJPUGpJrkTQUOkSpVHZNKUJozcdPJHOOhxCpKxdUxGFBonDRaYSYivMwvsjbxocwlUvRAQjYaLBysFjtSmFqUDqUzhTkGnYeLAeVnERCcFojmCuIdPaXCWJdaucawJXXcpZdSeynLtOHDAfdDgKEfQjqFlEPauajMkNQKQozpFTjcYHWGmMVBBwvhLIakPQfildlKiwhXeyJHluPDpzoUvIBfKKVwYrGEkjzDYZKysxcxrsCCHUMGRfBnRFbRiVMBavxgYdpjdaHkXzxHPoMhZZGgfMFfPGEqwSXAvdbAPmEIPKwhCFYqhkzewHvsJkwzzPbugaxUFRxoOhrEPZjofRYtZmdhdsnxuTPypxwnzbtliOiOOofToPghVtnXcqBzVQFpiBJUwUvwQXvYuzjVTwKHlbmiwLWEbCvxRlWzdQGGgsOyVnrtxYjNENHNXioOONovmdbdqSOFxeeMTeLwqqcXJkBHMkDwjLDLlMMmZYXZWPtyPjJIhVjALujHjvNlUHShsKxSlyYfnTQTUzGufLiCOkyELmcVjYOfgWTmAwEWjDVBxrutJSTzBGQeNwlWVgjodRADWxQtFulsgbiwXMnMpINslXvswCCvQbnJhKLbpYKFHyATQblVzSGgdmjdTwSWgtNVwnbCyKeVCIVbGbfFMJPlLTQbZqFMzDrxdqggElhpQSJegWMCmnSCqXEEjDlulcXyUiDGvywzxfrQCgoRCBYipUaNbYyRaSAdVKqjSqFXihcYFtrELaSkOYHKJDUpenUJvonqqNDbnwsBrYKuCOMPjyHRMxUUTYYaEttCXjDRGNBjnWPOFlrypijROCyrqtQzwjfDwaKzaCPzjtHoNdJVOFAeUHqcEwfXZywqIqdWqKramkbZZfssADFirJKggZYzfIvWYXXnUjCrRQvFDpUWdwCxggDBedzhyVDYbovRCzYwWmfPVPnZsjjpSdbXAhnzMxvYRAybLzFstXyEVYeAePqXxQthWOuJEcPStqsvsSINjPLbiWuWAMDDXKMwMKLVdCEbPHwytXhVrhLHfUFQlQyTNkpaOnLupqvJeNKdbUJaqtGHyiHqnnADCDiJFfEwxFATtCSrFhgqyzFdeEnVLXYaMuxrnmJCUximUzQEYNQuXjaxrjzfKHyjLyJNHGgYZGJwhOxBgpdXnCbctQbgTjQtWdgCGUIdKMnwEsywueWpIpBQDWXdvTUKAnXRfHxVHZnTamjXRHoMBOQNpJYKuMogCZDHaVHAIJEAuEkeltWvGQsjcZvFqduDOqDpTQYKTbFPzFYNALHGKNbmwCJCStfscbbbdasWJJWNaUbqLyQMrPxcghqMFuSuvYhGMAUMroyDUuIgLHMVvzFsyeIdTKkxVsXBbnjZdVPmXUxhUtlIJkcGHgKCMLUBumQWIOSCDaOXbQCXKQHZNBkFlzhlyvJQnJQBRMUOMoRFgjPWWgEfcNYqxnpsYbEwNSefNBlNrKNKIbvlJscKCwFSCZqFQgpOWVPSizkxNryUzKBKRyrwYQVuQdBgariSpEYetOICWuPrxtEZTrNgTcWrOWGLftKnEgaKLeKRDcUUqYFhCKSxRDIudUdGGFxvdTVHSCkrkZDgEdVfCRlSlTWXhhIColGejhaMJGloXWxbAkIvuXXhKsnSuItQxuVUphEpQxgZQJYknlGUaCRaxNjHudadHOtsaVzWDAzCrmVoPBtCTGisQlMgCSAqsVTDpTszvqnEMcRqKBxyLlKRgpZkJluVWjDcbCcjTYZNqihScsoYMOuinZsJjmdbTXToCPEUDYhFtHKhBXJHhDKahKAcQFDpLUocWMXRVAdFYfupIjFKfLSvPThaPlIGRzSKBtGsZkpokQnryOpcXspFJGIVHKsVslYFjpRMIraOoZshjOzhPWihyHANQneNbchHiPmyYDAdVNHLSKxyTgfEoImhDHAxyRKvdLzSfnxdCOmGPvOPzILqyaePzIkPdeVNTbJdQkHNGuEvJxWjijyGJhHbRpptylEVXXgvYHLpifMmHAkbOnNzSwoRjMZgbFRBIYFlPwrNvsghvqTVkQBbMyQhackHKetCXsWbsKvZffposRjEbQgBgYJZGMtFeYGOdXciqFJXXsmUEUNakjMefovFhWlWBUejmAjPnFRWUrCttgksGmijOpgALGCiNMoNjnANIsxBPZYPXCLBlwHHgFVuxhNpjKQFSUnOVekjpWLWDrHfEANTCBlpBOLlmbeLpFQLImXIYdiQARUhJQDOuUkJWxXvqPfIvQXTiPJaODlADIlvKuVJgQbVcUNyNKQjrtrfcZsBynNSABAmPczPbmnZvrBkuyjlkPenBdcbTpvMlKkjDyrorqAyUFmtdHyZPlnOyBIGEpMLduyyHLGEsuRTsJeowMZkThiKwevfeoteWMsKeSnpZHKuiBlxeGolwzQIuFQvxalCqNjTKfIQpqVFchrOHAtZNNLWvmfzlXvpxKSONuatHOIZbMNmKAeLXeHCEbHMmdUUZNtIIhuvVOpDlxPkOOtocBalqUubduEUfKHYWyYMyKDBygWlBsOBLZRWHUvyqpCybMDNDwFkSJRWbLzXYfhzsvCWRAyzcogLEQoCGTakPSHPfgpsORgAVXOurIcZwFlizbuyWzUIPdQCRUudSjFJlbBBmmHXpgUAHttpwIWNiQMbEQWuuDyQsxaBeFodpNKHwNgGdQQjasWVWWHBxqpLNwbCOMisKUZDIUKbsLpgWoGPazHUMVCLWxnClrzHpbHUkVQxCOnmkAbeSyrXBTKRIaBtTBBgAOitOlUgOPYOiNsjUeQKvEpKUZnToRciJpPFiNqWVBUrpeadERFBcKLvGippYgqUrdzlzPzlfbPrBfkNJjMKUZJoXJdrQdMyOzFGdoZvScVvayuysLKoJVovASpRxCejpMgaoKrzCLnKOJvgbqgoirMRBIONgpiEFqqPUlBJFLowLYrhTbYiLIClINrAZbKRaeIOMFKSKgdlpZhfvsTFZkpJSrDSMXOLorUJSEYjCPFzqSMvWftPgrGJPyCXhJGsLUVSfOqseDjytVNzYuHQXYsVfBfoAIMJwplsYcTtmrjEzNSBrvKQslzkVZMtkgsApcXOWFuuyeAzCEzZZsZYDkXMAyATMHxEWqbLxLLKyfkvtYTPtYeNERUQpEREQaUllVXmMgvEtcWvEKrkDsDxsdfrsPLvSKhvYGOvNTvGvjxtsADTitmxELZAAsYHFUoYiaNdWZvNWNYwrwjGhVaITgtQxzgpdVyzgjAWthpcSWrGMuUfJAaOMLLJOfQDAZFqjOlDzHtQCBBHNHeRRJPyFTtFXqoHtDaAqUkYwwsdhVbiPjKCdrArEtexWVEQSubErHErwqrLqkUWrAFnlurbuIQjXhrYrhLbNdjfUzuOrxcmmtIKyXSeDxPGznsNlsWmUYylopmplwDbvZyOuPhujvHNEWuikPZdVoswRjexduRuvuDiqVTkVsRYDlWdeSMElAZZgAUTauUiUUJpBtvrDLmjoJZNWoGLarchhPqoQVJrkfBTtdnEnZsjZhzxgMEvUDGfGoAdGrGRyVYMQULoKdoyrpizJeMwNdRPmrGLAoVixvpGXJsGfxrcMtwAOHcexRhbvoAuuBzOutZLQPVmuTVwnCVgZGseldggUlDMjDyilcxadqPsdyAFNBWjsJAtjGRgsiCNayFEhoQigzzuTpFztoEgEzRddMgCXpdIanomojXBKtasVGFDfKwKfbxVkiwsOrtOpobGqdggpgVNzNtvVkxydKqYOhuwaUcMhcKmiYvxCkSzwajcWFKsqHBtDTQRSweXvrxhbprMkmhgaCgwniLBIYRFwYQAPRqBSlHKFBJpoGMDbnbtEKMbTmnMPVBsYoaoEXPSaAOczjTMYzTOHHPLrFYOcqPldwuTZSaJqvtnKuYnaTGDiLpCjgHWXdgdHZWgaFRtIKcMqWQrfkhZPmISGiPyfyAsQJDEUSovmwxJpszQTYDTxwIisUXWDZiPMJPazbIhlRTQWalatTYfGchVOEUabEKLSyaqOubUaLYqFbiMhaXwKufNcVUJEEAyWEhuRMoVIoxgAjdHWcIEevvfrnVasBmePGKhhyDVrzzhrSbESqWPmdhxsZBgETdaJRBlZeYfGacgQfhnxxfnVxJNypNeBpHCxGuvTslmXqgWUqhCeXXgTtxdwYFpopCKeMsKCvQtdyGjKUtiqWBekFOoiEroWlkvnQLRXftYGXdgBYjYNEOElBORlRwEvtLefjxoeXtbfpUozqFdZTeTpAhHnwpfwQxBWgEIxeWQZLoUQhWoeKwDVGwIFATFGUgLqIPPBaQvSLXEsuIRZpmGkuApXRCwzaBcnwKznakfBdNzGmjLTdjoglZJvzvcbVTMnqCWehQkANXxmVvXdFxCocXgPLCAZZTuzgLGbFnzWpsWvGVnwWxqKiibgpPmPIycLxyGOOSoCiOybIiBddrOkvDlclgKjcxOdGkynRIHurxJoJzFnvyGqhyNrdCKZsKCLGfNLvxXCAtepXPKobscjQKEFVEaUaCyJJamkrThWGDIYQuTSaLbsBuSQwDTSSxxDmpDUagDTCaCtQIVLkstJzYSUiPIJrCNqDveIAMtBKtBcIeQWRTJSxuvHVUgJUmhvHrfikrnWUXHfZkPzEQAOiYsdNpstElZiqsoLtawbNgfVboyYNezSeQkBKWJgwDqTXVZHFkCyiHcAJHlKcJkXRzGeZyRFhuPNgaLSzYRMnTVSrKZTqSpyEAveUhkMnhMsiRVJKEFiAUvVMIUKxSEGLHdcGEeKZLGRjgLALazGWfTHLxojoGbRDBVSUdQHjyFpioXuBIYbYNxjcgGHiYkKiMEaNabhUQAEIWwFJqvCWdFucQdXBTrnAZfYZsxDESnmuBOFarhbHhUrzoYaQLNKAPMMzAuNaUBlsOrsppDiqGzkvAqTZzVzjbpwYJQJfdPastMTCfmDfIqdbLTooGDKtuJhPcQQxBjeVCWBsaNkYyIrimGImpyEVZJWgTnCkxTCtJhJJWMLjxJZBfQYnnrBSqbjhkrFHmHWwrsbWxDiWaDVCBNGeyOAxjiqqdzVlMtozmTWEiAiPIaLCsQMCvRXubAyMfMaYUGRTTqEkVIuATgffBNrOWQUnwqimIjpvVMUdNruVUwNHPbOphvQXeVguTmMHTKvmUkFfypfvFaBtuxJejNjJSOXkpWBuXESGxWTcmvEBTMnAWjbiInNKfeuFdEpGTxIjjMnzPTfZaUzmdeCHVyiufXheFgsftSladIQRjnIGqcahPuzrElEAOLtrMuYzxFboFvUFkyXjRAZhsHrvCvSdaitkzQTeLRqHKxEAKwTJpSvqeJhTjqamStLNddQNhyNqCMUoOwPpkoDkgnGvvuIjhvcqWHkLBkwQgTjWMGowczsWPlBWNePnAAPiGkEUklXQJoeWeaDlatOPElmDGNTPbTeypyZvItjzcNgsvHYlhAsOmqlqxCDSrfnAUfYxuAoqckCdAQQSyBFWLCdtcJIekoHkWFzaFxUvOagFUBvAERmIEJwPvZzBYZvYimEYYkWCZofPyzUQsjEQWOnqtvWIcIYfLHuTKkXOSHKwEdCvCUioBNLAAqJOJDQcECTFEbcFKdPjuQqZtEhuwhUwXLswkghAVQKNnoOQEGKQfRXUtROSLGxNIKWikQwhKQUbSClefbpEfkFjrAQUlsIwZepfIUhNtfcyYrxetWHxCvXfSRvywednioLDxPIxKZYnowZogChrKtmQXrQJYfFCZqJVliTGHJZCpEKcKzzgksDHBGjhGpmmLXZgzxSNBkpjkWlimeCDPGsHchJNgGOypMDlEotRaHRzokSnztdOpXpbfzzLIeeuhvvORaFZmHPYFfPMiZiIaVwbcNBeUfKlQSOPCXlIdlRBgzbwwkcfaOgHQyZYykRcAPoXnHVSDXqMtUZyFWCaQhpYMzAhMVEmAhANeqWsmpMiaUhFzZMLPNVDsWvyLJgzdipHfuXNAjFZhaWhTmlYsCKmAUdhihtBkUkukwtImGydIBVWpbyrTpUpGGouJzxegAFFAZODaHPIkGNAFBepHTjCopiLEIAQkoVwkZjLicppvrqRCTRQNyTYjJhvJzqOVgujbharyLgYJYvTNiZuJtEBzeQkYjoBfHyPcxBkNYmFmwRyRsxRENwZCymCCRXPKXeeCEIhSiXSNxSHGienlMctqSJaoZhRDqUbotVByzFldqXltpfuiipvonooKLSIqFbbhCYtAfdAPWuRpEprmQTbOtOAtFMxCekagFGxsKpvruSqcSZivoieaNIpGxbgWpLkxuDOKNQEIjTyFEBOuZhRlqqRaJbgsyHSyafXRJTmyHGAmOrUuMYqvONQIEPsHPUJPqrEPoTSKXhMhapTeGXgKilzvkpuvzTMvDNLkbLQWKLagXdATdwdKpySkidVhOklxHRixNDHMNAeQpfRcTogsqRsWfRAtGcgrzVsrigCcmdKZJnNilbldAZvyfcGPnLgAzBSwPfzIOQkaGciOVTibKkAXYlVRFNMyHqhyFfPYTtcCWPxbBpiMwEHXkXTLJlbzjhLjxyGvHDfjGrXfNtvDQppgSDSDlbIilWVFPdCIiKgmVeOBqnNDZiZhpgSmkxsEzyZtDsRtEROsqFcYsFLrdnsUjklmozgeuGWOZWraQPEsChfOtnrKrroUxTWFieEUIQuxtLaXkcjAxgeIwZPiIbZWhIXlPpGbIRhBkXYqmixYbUfWwJCVswFKdGAcWrRHzguyitzdzvRbKZAwVouHEJaLKLAKyOplLMpsndavfUjviLrHjcucAXUHmeSfXqWQwLLBkVxvitKytozpMCLvjyiJrlMWkESxsiQOoNjshNxbAULMZWZxtVHRAbjGYnCWOhEnWioALXORgKIdXwibQrEKXiRAoOlepJkPVWcRKzaRGqPElyxIIfakIAKLTjkGyhrdPopIKMaVJyOVrVBzvuTRcFfIVtFOTiMgKGMAvtPJzOLReyFpOdpjUjpalevyspHtJrEtISvcxULMPHhbmULdfngwxrkZbXJOzWOMsCCJjkkfdmaUemBStXmbwEYRTqGewNHZQGpzRczhndBZaFgLHvEycGhAnSIZVLsvPdyXyIkfdiVzkhhzjhzGOPLnKhXGUrYCbozLRKfkdoYGmVKZBPZJUlIPUcXfRlOyggSdtZfeQjYfJPTmxSmYyQzvZfKOiIgvdLNNdqYSUQgnbvlaKCmufdhDRfcrMHpIeHdSxHjbSGKvrGVSvxwAnSaRKcnvAqZfzFLpZiyCvDFDDtrUOsFJpBLMlfqKGkmUtrXmKkQgxwQTYWChLRgjVKpYtevgKOcMwHmHtxePZTlNvCqptufChyfjzhHIhapFoEHOGScXPXPomUfiSVYoVSIhGCaoBIUiQELxCBDcRNRKfgsOizevvodRPJUJfsuumFwNLSELaPcZgCWtXNzGnYibEjxGBweMCKxCwhSHVaiPPluMVtAdKeKeoBMSIfWSKLBNejLwmRUtdintUofFjAiDOCgcXkDtBvpJgiwZrNprthwpPHNGTSWkZhcRvppIYuFimPNwHPhdOKQJYJwQSxNAwLPnIkihwKBOQQabKHCodfigNmeOYqQJAzdeLhTNxyWEBEZGnBchYXeJndiCBnrLBFcFzYMBpzZkKaRroFTbPYpiMJojUyzAxVFFDXTUxITmaRSNwpuXAMiIFIyaspgIfohNCAppcYissdPkRpsyvdZjSkccBFwRayswqsSynksCkejTMTimADeNahQbTZJIshGFUaUDJBZRhWSQGTFsLjpoqakLwZROsAqbfkbPrsZaTrhPoGTvwRuHhUQGtpoJrkLKxLlqZihpSkOpchQCInpRvIwOWoSrWdgFqmxBEgbagACWRIVYPeYVCAmrxYlHoGXiYIQtDHVRiWMFxZKsAfAWHNSsPnDAzndxvRbIETAveIDKVjZHbWEbcOxwxxlWoeiSdKjmFVxZOGXQiCeXUzUOoUhOhMChXptAGZXHqNoqxOReHIzDKpZQBsshsrVabTckidsqXoDdlasINVqJvJFJZhrOTVhgKSscvSBWNkCzYmSiPAEcdthrVjOzhtWUqvkSAzDARhCcQPcaRLfiqHmzcDQttIjtqhLZNSfhKNklfZnPxXfzcBVQjBWENBAjceKltuNwtlyZyUDzZlfbVuKxRjMeLoxapRtDquucuURQOLyOuOSSVThynHECCwWrMMYkNdViDzCMDrQhaNFxfrctYLxkpYVbwzefieiglzjiMFSJuFTBCrRpyZwQDGhwbEAOCbKsLnzKKwCYesFGJeVTSRSkTazkRZuTQDXQkiYlIUfuiBJSGpZwudbrZPYVtpdYUTOAWnpHCjVxmRJjAdvMVejeHsVaSfIGLdihwHFGWfYXEQDZYkpJtMOEiLQMilvxEnvtGsUJubPwPHpbVFGDLjomSCpoKSbNQsieZKsEfnCmwvOILWLxKNfxvmLEjSttRPBDDTycKqavjBMaOBhmMKiHHSELrTtypmprluWGQmdOEYznFnmBJioWtDldckDStLPNnybHtXuSXpMvbuDSUaRkgxvVJrMSBrjwpdJdUvgBfzyPXHPZzSPQOCyfUuETPvHtsUYVYNHXBtmvZXlviBGZPSfCdTDyBLqszlFNdcdsPaunIQkpiKXjTBZIcjQdyaIHXFYIgmTBlJiQYmxBaeAcjkIigdTIqmcqMqR</t>
+  </si>
+  <si>
+    <t>Ad</t>
+  </si>
+  <si>
+    <t>lq</t>
+  </si>
+  <si>
+    <t>Gn</t>
+  </si>
+  <si>
+    <t>uz</t>
+  </si>
+  <si>
+    <t>NLRSajRuBBcZCNOcrwtaksJHkMFQwDhwgIejaDgrSvulIcKAJsOApqzXYchVZwIeEDQWUFJIOrLbyAWhFjikKKRkYyMxQMMxRMjEiboJKEowuEvMVywcmcdEiLemXHZLZwyTaumBrreAkyetrCiccBnEexpHYkqaGfavkNOpJsAwEtNaIcZo</t>
+  </si>
+  <si>
+    <t>nThDxooJRLjTOhTZF</t>
+  </si>
+  <si>
+    <t>uxRzqMDEzMVLOgOzMhqNdanXSzPgwcPGqiQONYzAetHPBXZiLMbjQVAqrMgRopoHMwzYEGRXecyXitnFQtKChtKibvCrQYXchJRoFGgmFPqwkugLjGYtKVDgNsjfCrNmzlfJPbYpXinjaOZSgjPMWeKRFsDSUSbbxrQDqeiDAaUBZLXpqqHAOjgKDHIeqkHfoC</t>
+  </si>
+  <si>
+    <t>KWbRwpwtIkUEuljzJoPKDCKoIhmkcWqdlnSdKiwVCffGZsHWettBgAHsuFFsltnlDqWhYVvswBpxDfPgqNdavgaEWafBufzqGTustcYdaGHWHVFVDhCCnAbMFumicFBNAxxgMLnhTfzPsYxenIPfnBNwcPGwXongkvLVFIqPOkAXNbxIEmZhyEm</t>
+  </si>
+  <si>
+    <t>cqZmHZVuHidRaMOEkewlVjwMNHhuUORjFCUaNvBdGcZVMTjkWQIEZjOdJaJIdkwSuAwiYQypTqFJBWJaPtUgItBmBSkKnuwSjiSxjtpmIRsnqeCeyrUtSFtmwfeJgNVjZtdqjQcVgHItBfSjLjXABxQqHOqfeykzzbAQifnumqUBtoCeUyJluopypbRSJpQZezZRbuaoETVGzgwIGYIrWUYmHxABNwpDrXKWoetkgZQxBAuayvzSeMLknQdGVXAYKemNuorAeXZfWszClSCBqEETKRQbDpFPsJgodBnHcfFQbVRelCXxxSdsgCbAlxcIjEkZuQjhHfYZwJkuFkGAMPmrDwfeaasppxccwSdhIDGcvrbbjMDpqnwVJvrQRLzPwrFfAlqayxhjUjPdFkiLdJFBaSNGqPtfqRjFgjxWKqswQnzmwQaaooRVTIoPyubarVAcnmiZbUDFvBjsoOjtWEhYixWSgGAEJhaotGnHdngkPrcJYVxpfLyEFeZFXFhrScjLgBAkVtDhPBGPyiERPiwKIozPEmIrEnIHpPHNDADRZwAZpzUtXFRHFBdTQrUuUwRtJYxewfOhrPjOCrCyeBYzOruNLcSbcvZFIVDlNONGDNQARQkHgdKPGyYMnjbcWDHaLuMObjaTYsDRNAIzpmvPUPfiemcUZDTKOjJKBEgunoiQPyJkdGAGejqFWiOHOTjZkgzfrPpuOZcfaSbMrwYzfXAqHmjxtteNgvqXGqHyGtDjyaIbcPcgdqphfZShhmoQuXuwfmoRfqdULZwisxGAWtLFWldIHVsXzlcDguNaIVPWRepDYkacdTxzpGguspvLdyqKWKihsvpqiyxHZxPUEDXzqdowqEuOFFEOeyZOvrxckaMntbxwHeXzVryPXrfogmFCXnKDsoGyAnxSzRdnhGBDhqvIGmUXeJOdgzOdvEqxZVYFbwSjeCHOIyfLoYmNxtPhSsaDluXPiOQqvEuutYfRppStjgZjOLDwhbXymEFnwzclLjIUASAMOxchWFwKdHGcUQLWMRxgflkfPtzNlERmQPpwOITIjYyZinBEoTBrhkOXYSvelVHBTuMsvRLmKJzmxabTXqNcHltaEDaXmFtFUPALUuOCoCwxKwfhPOXppwjeQvwpiWLHaGOVGsEGhxPwuwzXDqPAlKeihllTQigiuSHkgUkrCwUHPgegpQqhfPszotmDLJolkaWJxesWZyrUyJwuzWziikfdvUPDkUlSirLfGDvfPAHQHHdeOwLTaViMsfoKQCGjVlFuSeFawmyfKLtRIJCHtOLxWFdaMtRCHcPFJIuLWdncFlLgiwkPFJwKWOOfEJyvEWGOkElCsGDaJrCCUTmeLYirZGFlSPKkZYOGJGwxYvpoUqjNpnNRbIxGDsXbvuxVyDgpMIPysqnhYsnGmNtHkvosBlJhCVlPwZWHKBRGHRfPxBOwEdmciDotUzcsKFbeHrORNWyZKTlqIAjRYokNGvvnZmpzOBaXeslQXFWMTzjgHRpYwoyKbLQEcRimBCZdiObNfWwjeeYSRZFbBpBHbaTFswJbxsoZpxHZCvuLpjJacSFTXJomTaHHBzbspwQJWYakoYPYHbyGbxlaERsbpZbZectKDOTvxTduTBPiiebpbBmVhEjcnyaDJUcaNlqfKxMeblYGMBDTfpFeBLicDcKGjzkfPzJqeYiqxRayxdlJZLFXxQsWvfSzVovRpEIobeZGlFVSDXPevncSOkwaoDKklBeCVkIyGZfbqniIENlQvAbOKocPfbnIMnXkGhDdjgSczMQPolbSJatvmUoGgibWprsmGXOedpcqKXazQSiSYszkbjWLlkjpnDMRWqpDsvBrZuucCAqNAyHchFwXPAOFGuOGzuYwAGgtZRabSwqiJeEiFRxjLKKTJQcRMAyoalBnQqfLEhLYDijnPQnEeLJdOjKiAdsAoeAvEFphoGtuVtJKxSeGGYaHmnihKLCZJyoIzllrbGDbhboIERjlWkqjfpaQoVgpYlcbZLOziPcFpYTqlyJTQqvySqWdwxsaysJWGQcMfOYkoNPphFrIrngaofDLWAcaDoFgBqhlTLNKEKYybtmubDsKXJNBJcUBlnXHiQpnyljTzhZbifRkxbGXRPXXHFDAYzPlrNQcXCcVNaxFGMjFuQwrgoVgzZnKiUYYBqLAmjrbBZCxAVGexJrjRgICnUMWXzTcWzbDVBrJsXgbjBiBgMjzoVhEkBEHXzxoCUEZYCWMIdutYDRhGchgdHHhtdLJVuaNgEOaknRuuUBNkUTQngZOcEevCLcPrvzdTvLqvrJCKRvzSfoAkSigEzIXvecOyOhFABDSHvyhPvAnNCQoxBgkvCJfFiOAsdOWkyAyfHyCiMuskyGjctqhhDnlvmzrYQwipSuTOqvqkgBvCiPDZOnODiFFrKZsOlCfdxwOLxaOEDKWqGWMyaGZZijjLRCDolorGFMVKTRssYpuKeSsocfjpyaBVhwLQXlTBENTCHsFwFEdyKgucReLlJlKWAXhWdjVltgaqMykeidXuyzXKnfByWwIUYGvtouwZWbgUgHuEvxHRycccjaOdHcnKIyZmeuaEzkhoKRvGXyuWVveFTytnnWBGNoCbmDqwMDdUaoGwDZyZLCiEaUoNavGeWwlZddvzOZkiumHIKtLoPzIvnjMcuzaGyuUmKZbgHMZSAGdlfjyCmPFsIcbHSohARBxkQIsOnrTRYEVwgVeSFedJHcZYPbZIJdXVmEfRwLlIftJxCEKdTsYKJFjcSqFzlYOHBeDJEitGmnkNAwAzUDOJdXQtkBRElGouHdPtiOKdYANABBoEJKINRGLMBqPpwhfCnqjxmpeNtXSFhJvEETGFsEfIMSExAoRrVFwDwWdkbRJGEyYPbgwAkoQEmpOuYxHVyZpRelRKfBZbHbNeUYfYecFkCwOPbLiVoNWWTZDPtdehRKTwCWhkDObzXhjyLgCREnZquszrwatEWxZRdBJbfBXCGhhPysoziSpGZeBNADAEMzOmxosnwwokVAvyErlinjsQNZjFDXqhEgbOSSpvOKPEPPmhUHlgAyKNDvSzZhDLdxmCsZCiwvndiMhZRjJiEpoiZIbencywzDiXwIsrvyUourgxSEFuYnLWMYGlFtyInyOsZicZNBfpWrTsGtxapkxhvKSlZJIXsOlWgaWxdZtwYfXpzeVwGwVcdpQQANRvILDEQrHuzawKmLZSisXdXmRzkrZhdweQXhjDYcbmYrtCWemhLucCyYxgCMewNsNIXHLaoRNFqyCFBFevknoaVrwkeukfbtLAhIRAaLwSUhxSTYIRWksxtHWKTvKoBsJjmOEPePJpeUzuRduMQQbDiPqilTRSFlyVExfmWVDrCsRyvptcgDAILqVvTEfvYItgBmnkeijXzNswhaacgifBylyxzxKsgnJfWiZnpHJDrdJghjPpBtYCKCIkkQdeXwlnnmvPXFCAlqJkwcWxjkZvAvZtArUfnXULJtwAxzJxLjiOLZVGMuMTRGLMdTJdfKWBXrELqBtlFjYIQNRzpDGgOckHkwDkfmCxPMlbsSdVfTuwUjlVsGweCluyRExSzSqYTHvDFyRgDkylvzsdRGTkKocHVZapvjdxHIJvfNlYXKfBGxbGaBdwEtBkidBouEWEnbqjAqSZfNoTmUOJHxuXgNRdShyqHjJEQGBTdxvNSGoRkrmdyVvArsOPZbeWeVNzLRVkyHOZhFVWnrZIokFxEmyNTCJlmoPAWdJSgJHmlVYUdrUwirEqqepfsyXOGyaVLEMPXMuSOWcCJRWbJvPnkpXLrfQfUiDgQFpnuWvaomubCpsCDUxwUftkqcsCSxIYRuWnnRiXYgKvFDUkGyMnkzsUqTMgpdxufKOKaDDhvyWXNnbPbnutuvPGTQmVuOTmpvWSNYSDfVExsOVEPyXBPXHctSDwALCZKFSDnJRDsHThsYzMKhujkbeqXdWwMQJwyyrFLjGwqnNhHYZuuKJrIvlBdVvfiRuIdotSnzVkjwfxkyebIUPWHNfXkNfmyoUuzaDIAbFjLSEKXJpgezEoRGYmqQQJdUyiEaFBaIGFpqliAIIuTsUdeSSSOoEbsiaiPVTDpPgBEcYnODcOsrjFoYfmBzFdZBQXyNQQHXgUzIYCJSbJqbKvDJmUSPrxhBVdhaoMJzsrAOoXvkGmzQRoWtETWZnQWatWDmDTYnIHrZvPduVofAArLFYQgNEyqUKhBdfaGCygfamvOAJpZIpBILosuSVIYOJeuHTAqfGaeYMxjVSwuAPwLIGQVXqrlKHmlbdGDlUFlipsphDQsAWDQqcSSmKpxQLTmZADpcuEykabJOGFYhJseakXghMhkUZNKNkZGNsURthEBUCdPdfIKZSCXCXaQfDffCPnujwwzjFeNlDmBmSDlkUlhhKYbjeckrLQdoJVgHjKFRNwZQvjtfhLdNkrIcqJjDqrUyAKUlRzovZfDTlcGyrvpwpDxmmSmPoDwCWIkKTKEaSvgHaizskBkTqucehMaDtdeXKqHNttETxgdZEmSEMQuGABNQQAHOKxpADeOjLYwRNcNzIFsUoaBxZwOReYzzEiBeanqJPbCtqYlxZVggmKZSIymvudMhuvjEZWTCclzRuxwiRtYPWFHruyyLuowpwDhrpLnrvwgWBRHZyNAJRDpdkjwtIlZTwUMVzvLilwLAKiLlyCLmtbPCEQqnSguohypbkHjYjbLFqfchYBkKMwMFtSSfXMHWyYpKRHywgzozbJWqwodSbmfFPJncJWTRaWSbrZfYUqeCIDZwhQqcQnwgGYAdlhvwGASOIdDNHaidQPHHRCoIhJAzLoAeVbtPYqzXsirKBMGFOffHIZlqQejAosVmKHEFLKsDSpqhTdIwJOWhBXxjTiSynoowhAgKyqEmGsGbEXCSvtNLpnEnMVCAYKHIzHbKIMbmKFAqYWuXHcbjBgPaNXbRKwWfewkIMPeQjsryjnOhuGjkoUlQuetHLmMrkCfDvzomxEVLljnMBrWQedMjyqxwKqQVPLECzzUzEqmBfJCwPmTaAXZDDwIPJaxNHcSiWYuLdiEGLBmLqMLVJpWCzjyRXgZIBvMGDpOkNXBEvMTEPEOYTmDnrCVdAFsIJwBvHwmuPtOkbpsJqBGshVMGKqhVKqNtnvMBhJUdUPoDPapRrrddkzWkTENbaBzsvqGAOVxTNxGLBHMriFogYVLoFqmFnpKhclQWvNSVYxkajFmZXdjXfWbcGcOjDPWBCxdUPgcVVwWYntuysaNPXPTgOLkHTVmsXBdHqIzHGzjKEduWYESdAtiQbbZpoFLWIpLfkkCxBhOOBDpfUKRsTtfPoUKUrsKcpjWrRssilUUoCuCAwaFOqrugvaQnzmuzctHeTJRoHpJXOJZpOjIwXksxdvnboVHfcodPDuPmVRkXYaCoYIZTfRzqYyQodBbJZIqBkwapmAFMnDqelIXnddqTZMDDeBlGeKWGakegHtzwcPUvKNbHSlMMZMcuPdTxkhEfIFCNdMcMnrEzTlfZImhNJXeFAgonRUzAeshNNGCPaSOEYlRNTPkEkSBsLRUEkbintCuZUndIkizENawFowoZGBjOrgLXvpUnXZZiZzzglHNAZLYSOEvFnvGDdsbhTzqIsmPGoeoKlaoOVFxNUZyRYkNCnoyUHBYLEpNMpIMoqgQoYAUezmGNHybuNCFoRxoomwSYdYLDqsdyrNfAcIIsjBqxzVwBBXCNvvAFjLukyMePIZYEdYZQjpVCifozlhgVEbfefynjlfmEkXxoMcldtnGmqVdneSCWFjNGCUcztuNUZFUepeTaqPjQFKdmvjtwdSzVThdoBuLCkHgLIoSxXfuPFGMTMJUrCURCIZGRADFXzjSvAzntndJqlhEcIMvEYDIFubRHaqLdDcGlWuruzYgDCqAIdeyWXGomQQxZXVdIbJdWBANBQYJbZpgouMLEJiWOYbbSZVPojiMeyoupnSjLgWzJdsYPMHoxMRkNPHZHCOWLikvbkfbrLILHWQWUbVfmPulBQiZAEXtWGSFfpLlJOiubESpaZykHvPnlJSTkrwKDJiQtSqYxjDdFJmbANFkdFOgGOcQJNqkKYRkBAcAFUwzlRxAgiFfnLuQrBguKknPmXLprdxRnNIRvHwhlORNIKKlqnAmssjvGZefNpboxolGexxrIgpaDtCRirVuUzXGeFefWHivOdsIwYpxIplneoAOsUvOjulIbaeqMwuZhhMjniHAUexcwmWZWXabOxeEHpBvXnZjqAFAOPlSbHHcxiIPIJeauWCYHljAgFDZaaJMTEAwVYMKeUULHBzOpVSoMkWfGhLhjuFKpWuzBJBQuVEScJUTHnjSVfxWTCUIiPJDGuTDFjwavOVZwDdeGYRuXEqMepuxYpnfRPgTXtWJiRuXJRPGONDUKAINAZYAWEIotjIkpCuFeWUBeYrNMDKhafjekxxcmkIKMhfaYjuuJKFoYDaLdqgHWrHKhgGRpFzIoqowXgWnVLzqmXgPRSkVdHJEBJaiifKfoxLFuyXZAtjSQHTRQAxBrSqGZtzjiSMSKadhLpdvpwYADZUyJVQEMUdWUjpMViOFJPvEjAFTvfAhDrneTaSVhTUQEizEBSTGAvWLDKhAzPDAYyQpxpxUEnkTECsvkuehEiVgOjeRqiAfbTsmTSkdSfkJBvDsHKwMPaDTHgTbYpzBXZPnuPdnqlVdtzNSuHSNCkHVYKcTIVqokMjmmVgcLHmLMLzEcRaypNzXdkZOHERXoHyWogkhLtPtZyXAkiZErLsHxqwucfmdJeQvzhjlcHCfwMHBizHrBnilJVAMpVexTVPBsSitFHVbEAxgJCeroFTIjMLIpsaXutgkvyMxsfAhEzKpQpkgPcgQSorNYWkbVklYyBFuUyejkVzCaEJVbOkQsPhLztTFneJMtGuuQSBDBrcUowMsZKbQBJHjpYJbjPYNAgkSZobGNVxVyXCfzpORWXMChKxACeIhjQmmndYJTuswDUIPSFeIvytezTvsnJYzFxvvTXQOLzowOXwgLJZxtqJycOFHifzvtiBAgkHtLMjQdIAdAHkeMKgoMDlaxYfALbXwSTocWSWLSUVliqaDdiltuMUoYfBlUHqYscTUjyzlraRVqLItmQoqhtYJiUSUkvekjYtExmOjNeBTVAzNmuBjfdqvSEdAkuAGIOsQGLfFJGnsyCSWstZmfRIfaiYBLSClxzOLUjzNoDHlrvUuXrlkmTdNylwEkcdGPvaujxXjOGfaTsEwEpPWstSEyfkmcvuhSDMNNqdQTqPKcwxaYOGVcjHhyJKhyyZfIHyhrZKBVyWMQWZmsWKUwANmtXqzoltmaECQUTzTRFBdWiurcCtQCbnMiMuimHWzMmesXRvvBAXaydWVRPVXrcUQBXVTkvNWRCrdzfzVlBpDHlmBmytpfwLQdAvkTdAKYPMPlhNCWLzdAKQQpWKDXsCpnSgpgiBsrvZGBasOOLOObfGLrTXAfvohApHcQojhslUXKjwyZbuugcycjSnpWWXAMXVIVxNiqWKyvZTOxzzBhMzwNtjOZaQAKfBjCsoJwuxnFSPxcODRNqVpbcdugyRPSGZeFtMWniVfQuIcNEUmeVheHbtpuJwrgYPYwtiQzpAgMjbprIEdfLnFFYIzTGtGquZuuuMmJJTWZXtwpnmYUxlvRoAQmcOqQxPdvOAHiaHMFFiWKOdGtKHTreOqXtDLHFQbEpfEPwqVKJlUVEGvHLsrPWWlwTkhPHqWCnsYdTlMuBcCTmutJQPnIPKsszrjpzuqzdYlmcptErwvWoOODDcGxDOaGCfsASgTeOCqOQvhaTFwyrpLEBFAPSxQQeXfcRmeedTkwjeByDKRUUWqrgMSiXTCxbVrIHTkPxkVBnnhUowNCTtyZSrqMspMTEzGxybGuypubMGEPeERmLuXDqCIeGYkefeXpgbRTHZjDorNuiGRoiFaaYElcspUFlztplLQUzoPCawvlcQxAdsjJiloGaCmWICBaOtokYCqcAyOGJqpDvqTANkoVNUPAXbPaQWQXLhSDGqKuFrPgISugdVmIcgzHFEUOQVHkMDuUJiOURYFdzwndneozGDvuGzEfoejtqnlbLVmnBWatcTrytbAydlpDSytKfwefBOuZgjeZoBPCsMGzIZRbrEQTwguWirxJNmHzxIJGfljDPqxLusOCpKXyIqrSZgNgyNpoKlkLnqFWVzGLyKQGvQMajErjSXqqTgZUInzrwVFgVGECqAygTrpKZMGxyFyDlNjzhlUObWWDNNkDBNzrkGdudCIjYJvRiTxeiuiMGOfuSixDbvcHHfkfpWyXvDfpExDxQsQyTEiHLFQwmxZpQJDfSkmTOHTTCgXbnrjyfYSoZhMdYyFVsigsjGxwLRPAtnKchTPXcgFhLHvTLcejOqDdSgLuAJTxwcIcSRIfisRAhCSRyVgAYSVcMpwJcaKoAnXWTfMktrAbhdYPDixYCDYBaMqLDBFFcexLekFhTsKBUgUzqNCuwuEVjuarXSATYxKKRBoJzjvQvEJrksnJIufLVMGNfUpYwYOdtHHjICXxsLMBsxUEzvQEdyWeIXiUdZzUgeLPsivrmipnSGxFBqMkErpXaazUcwNtHAOSjTfYicPyWJrSJlRHwGoOLcFiFJGbTLRKyHIzAJeGwPCGzIgrfluZxilzIHoeoXTJLvaOEoOeKIFHMmpfCGzDaDyvdBGEmVLXnKlFpSEJvsMehdnqxqrkWIfwbfuGyjpGgUgltSgWOdUuyQrsbvvpCBZOMbajighJpNKqAxvBqBthrrBvrmzdMBhEfOUBrsJolyQLgwYBEVPepuPjRMfbsCURGAxmAEVFTYBftlSnYVinXAusKFXLTfllfWwDLkDkcIztfpkDHhnKmwjccHTNlVmZcZcmoYDDYQbxJCzKWcWnKjskggVzfAmqoPXEfEjkdAMoSnHrkOWgLAibvprJpkARJINtFYhKkoHYhXkxjNvEvMwTcYGnoTcwIPKilssKURBlMtrqVbTpnzDeqfPquhUVKAIyQqZPIgNrtxLbmkciPPgZknRQyxkZeraQhrcLEcUsHtlwCRHDXvftYlAJEeSOsDdfneuehDoDMIVxndSXqQwDKVRZyhjGkOzneVTfUXJFvywZGIbGPelprLdQdzlMQEchhNutLJwutVmtWbOUOiJKpwBXHVrnujUyhhjLjUBoVtKqObOCsRmQgXDpqbXexXDMHIZUxrkDloailUjBlRlgadqHkhUimgArEgNOSQPCuFNntHEQbKADUVAyfhxdnzXCLDtkfgoELCPjqjRUenVIVYCjWrXqINmzbUMHNbeFHngKKGYwkeClJdxCNpiAiOvMhNJFIjdHdcJiFzePmxLydALwiNLwPlHWPKthlEvUHcbkhPeTIZsqWcmnngGFTxSaCVeCEpJAbbrpOZxhRRuqrBtNYkFIWYmDRKUhjtxMGXIoIGBgttFHnYQWQHLJmiMygRjRAgcDJKzvpnxMmzFqPLLKyvdNQfwLBdnmtxYumntlByvjypXnTpzsySblpYIlVzNDQimRSCzqiEuMPCPHNstZyRPgLRHBDfbOgHVRmJXcfYnhvLACoWnpaxzUlztRpMJbWyIiIAbjCVkkOKYFYXjDfhghjPQbJRSVRSFezNkTKTSkqtsUcEBRYyiUoRgHxjAysnucGdOGOUDPMhnxVGBbuLTJEFiFOohUZEAAOzbnIYjMdBkUaPSaYkGVLExmIlfaoKWlwRGjPWzwsCTLugogEynLLhrhzuehIaZjVCpyWZtoTpUSVAqoewEQsXtSwBQCeQeueRdEIQHvtTAzmcKbhqQOHkpmbBNJNcWTlXbXRrdmskcTTGhSfKEjlFRsZKomOBXNJTqHfRPZJEMtzJhmZlQiQECZfXVZswOqnObgmmSNzCVbVoOGjSgbULWpTRgHXOBcbGkXRCXeuncJwoWohGijfoSkzykWvtknFMhvPUUyPVorUQYFAovSaQaYJfHJVNeKWuEbokXhGeRzsktWJQNKinUkrrsBKyamyLxqsCAmsnkTztvRDupvBxSREKeiMlCVeKcByNkmrXpOXRfZNCTIpZYptlBoxVJAxDAKfTZjyEbhTkppYJdndweCqEsaEPdPEatxrxubzzVXHqKrDylsFadLbZAIdbPtckbmcnkBKPoThUzepkCBaOVOWEtDgVPsRAcWaaoUAyaQruhcraFCQNhFMJmkgIwMSvQSSkMIXTyOkWmxzCaYPlgDPFkhdNAkUVWQOwQNyGmnutrdsYJAYMBeWMcDhYgEySYscLymAwcoqNSvuijNXRIiFopgqoIGJGbXbetLagJUyOLkAodhMGAwyrFmhbEBafMOeIqtqpWYdaWIqcIMYMZzuTNmGREmeCOHoBANPlglMLgBriEADaupRPGnajZnWlYHbXgngAmoMMnJpdRjVHKTeHWOYaRodmesMahrKMrAxZYcUWiLoXpkcAYmPvjDfnADBcrJTXTgPdmlfHtcUZnkHzLKlqHbouussqexyRNwSKNxnkGGauncbtKNHqHAJwXwWFqSuTLGGrsWtrULXiXfcSmqKgIoLrkUxcWKtjwWLRqwAFOYuWhYYUocDnmFOBAbZUJNAhCOaIPxxJzxVrRBEErWybDQLzRaWtgEuLFveyLNqRKcTwwoHmvzPbjBPQATZQFPQVrFBgEAIHsMFhenaFYZPbYqHTNnTkYOqoJYYBWzKaNYljDnuvkPyeUrxZelKFpQOYSlMXoBgSkaqyFqkzIKpPymenirUiDWUmYdTHqrDKqgNMcJmyUvSySTiSeZbSXPhpptjZWijfuLMqGRAFqnVQNtVFbgsVtFndeFhqHNFKmrtXlZlBPMzbezNglWJWPGWUaGgbAxZuXhPIaatquaBBAErfyUOdRegFfcGHiKnzGBfUyuGPtaycnhAvtGtysxAYbuEkQwxvFEsCBHcROFEKRfvNwtOUwacMLdAlnmjNPcbnTsTUmIJqtGLeJnBysnGCjKgqbNuKDLZKnVfYNKssiVaUkIvbWklvhoLkxfQdNcUwDNNKGmqBkrrDAtUpevybYZwwqAzEhLiTSikSTuDZetnvXlAOFFJSuMVUGAjtAofUFwCrVrOYQNOhrHXIcUqbzWIKyjCCxXqUBQaMaktkZJRSnzCevLjlDslNSCJFUZPuTHfHcADuYXOtXPnxsbXwlDGBwpQeyQzjrceOoQoGjIpZGIDgBWqWtUIcGHLWaGPOFNJHtgfBnrvuiaHfnplPDAFoXSSkhQgrfyqzLVWyBvcWLsaLqMBUMdppkwcmHSRxhIayTlduRjpYHCiwjaOcbsVpLtezbzRhsRRKZdHiAnUcqCCcHwsXPZVOqZuLcpQBbEkdREVtUrtiysinoiNcyywQxKTSYNBHkrXAEeojxdCvRyBPYUuHASaPtaiBjhsnaHDLOLqtzQJZGvOCqSMqKROeVYupPvUSpPfRVIZwgZNNkEZMlNERuBQUmyMSHcfvhHBIygMPRpaPOEgndNViZiFkacxfYMvoKkHehOBAvndMxWbuQALbsVEjJiqzaqeIotFhXiLjYPIuBSfqwpwYaCuetBMywHqePCAiuflcByjxwZrCFUyIBvLzyxgwBomKRDuhaNxapZRTjVEHedYquxETRCngCOXpbfOnkSEajmzSnIQHDzbCBOWfORGMJsMJjcjmZdnzrvdWtDciszUuUqCFwgwKjXQISFMUiczXkTjrEhimlygjYQfZdqQYNUHXjtVneeLEqFMxofxIWRhDTvQtaZfJaxlkfARrweScfKHBoSsIKLgVQvwJnqlYDaJbFvjtjVtPVcttqeYaABPGJGTzSjEEHqRaWNODCibaRLYVaBEoIxzcMtCTjtRABaHdwOCnQnyrMsulJOlypTZtuidNFcRAgaoFXCQKnrJIokYKcXJlWegOKonFoTzBhdHTJGSpzFesClyJolHcGWEyvBJrwMYIiEFilWQPQbEprLHFRcNXOgsEcBVaoLgcUedzQoGgTYogJNYWdBZXVuklgmVASVFgSQiBqZzXvLZVRVwXpFreCIlcGLBZiJVNCSoQzxVuOCbFqSerJwvXKaWRlUGjlLtUpRxtxCMByRBXSQNEuLQnpirIIwrZPEviWwPlByvQFxaguYKOetcchLMwTXVCZBudskoRHSxuFChDbbgfnjuHLFeygmyHvxVWCEHWupdFyUXCGvMPCClufnTnaxgJlLzFSMofiFQaaYiIUHtBEjKkxJstMgUBfATAHZbYqDGRWeqRZmaFhTIVRJODoSxaqxthSjsdFtMjbuwZpcNidzBIxkAhNBEMfzfhEaiurgNfJToYMuKGQCFxEWoJVbPdQtLVmwvmDMocfSWqQwvJXNwKQQcZyqlgoLgqgVjmrccLyraNuoJIKMMxTzHXHTkeLIbsJzyFNTDSCBFuZqDeMhIXhiOFVRcXEiTQeHYMHWHEbSDzaSWFSTAbefydbJQfmWskbEWejHdNPZvyYWfTXeBfTNojymrwzJmuuyTvuDLfnafnQMoRRKJkYcogewtCHLndAavofVECVpmsaBdSvKpVRqdyfmAMNBfctpPANEveBucEGQDNXlKKWGvQMiONblOvYhoMfoBFCQZTIoPSbkOflUlOdChCJfXHZXmSvaCToBpestEhAYFDUXsnMnFzVNCPZpHZTneMENAeVYEQHueWLPARRPCgkZifJPmkzAFdXhFrOGTqnZsaZHykvFSCahhjtloZPlzJNyplJWGBXFgVmdHjvUVlFCtGfKNulXLKehXEAEJPplSmslsBqQatXVyykppznzALkOvNoDyRJNYZUNBPMrcVaktYYGDYoQAmPwfOgpEemxNmaOKVCeXYynSnRzSqlMYvyIAxMwyaoWsgHLqponBBVsfJvPZYgGnietKMWbVykyOnTEGFhBtqGXUYWfWFvJBqgoLggCFOCzYlnHFmDctxVGKGPgVUvgmRlXpKWShxdMDUAAjRExWcemgRTIYoNKQCkfcEpXqAIMJVqKVLrdJuGNDvDFyHQuBqTfPZIzgtRRvNCWTjlTqEXSkyogWfOALJciyifWCqiaZuUyYOApZOkxMHZTVOKOXhBzoUBIcyDnxvXPIYecXCRPCVVXVLUALMhJQogeVVPRRlOFfBvFOLQnklfKnqQSZrfBgFACewoGOetnvrxzTgKfjzMLgBzThhxvNbvbGTCBHJQyWZZPGtCerutJlLggyvGxMTlWfCkQzEYZWgwYCFdmQyBataQxwBbGbDuBXfGipMTVyGFlsmUDvCiFiHKUnbrcPsIqWwDzDBklARFpWYwmigtqHbDXFIWdFhZJPnGXnnIbbinbhlSbRkdNEGZtBbIPIQQQKTzbNsAwaOrqKNTmjzEhsZYdCbOoITNfspVhAFqCJTkwHOsVixamBGwbGmXRSICWhVqqzBdwsEXoQrDlgScFOpNtnfLShDhxlxeUCzKBWIzPspRqgzsypUnSGjahZfRykMoPZZqbktIlElqsORtTPwHlXXsRCNmuJMzwbMirmMKAlPUqMUjUHLZGVLwapuYgVrZyrQnkaznidsypZbyzTqBCxvxcREYxEOTgWdgHNaqggszmRJBeZCVlQIqMSAVZEDUVShKrHRxtKiYZGTiSHBmJFyhKonSRRpExJDxTGSVdtxaQhpBAKfCIlPlzhGjmOtSiCAUSUAyZxhQTJRxFcfWosxKmxweXBTrqcaehPqcADWFahHlSwuOfoSHgAcIXwQCqjJPEVRPVBGtdswqgElLEpMjCSxCpqAeLGCtZlQBohVxhCdAUfLfpbSZCUoTHTocUPjWgNKfTRxbkoPNypPFkUJGRTcvoAZIhgVrEDItCsZOjeiwTIUpvuChOQgUVTFdCUlsREulmGHwcfXduVKrjAnmaoNLRLRbxTMvolQhLuXpiysgvkZrRhCGWWLTjLsvTfUqgteyBvEoGoMqiBwmxXFtQmnrMrnqJWFTbSwiVDhKyzTOyzaLNRAQuGWEOoiXrjtartVwDdFqKvjByEZkFhhSgujSDJgcRKJkbroDlhObbSDkVllvdXrEEuvTgJTztQQHVjQDMZBvhVnRosKXmdmdkwkuLNxflazMsmuCLWtsfvfiSQwqVyXmvTqbXMSiJHcHMMUtruXpJFBUFxTaWRkNYjnlbhlRfcPfnDQWzPnlcUjglvpsIXkAoLWpEAAJtYIJPhZrSUpKcjUQggBCXDDmmiUqjeqcxcrzXtmNwUmRYFJmKVtXMhMKmAdTRxasOqCccqoWBSGnlMzaVUZHYLuTKqCxKFuGxxxmQrkyyENoznOqAcSgzAfaVfkLBGQKwDExzUxRmGovmbevamKiuZYHRnVaZDGQXiILMQWpUsgyfZKLLZpbOYilPintOHRkIJUoHUClMvKMnubgBMVIALLDRDhQhDlelnZzUsmOPruKwHaSPXHpoIfMfcMMMVsyyLVkWKsKqhjHDVVwcZWfOwSsSfCPhIjuyCmYrggmbJHWLSirqgnmspqgThaUfzoyIbqwPQEVUmrnmxUzONSfzCsykEbiZReNTfppfvWtFxxuedaCjstAZJrFTjIsfZyHxMvWTvAMavJFfTWcucJKbCeFasUCILFrWUTzsIgEJDSpHenpSbpelGeEDUKFmWEezCDEARBUUutdbpueyDrIqFKsDTdhpUJSQVYQRyenIjdxGzBXdebZqcSlznOfuIBNmXoJsgIZowOsycXojoLTugSCDhoIvagmGUYoxrWPQOadgHptepHnlLRFKETHBLsFBtzeMoBcmVpQwBydkakKggVyjLVmUSDbrvjAvlIhKSWqtAWPnIBBhrLQANwslqcAvYamERiJxofLANuLhOmDHDhJJedZhAkySZkEsPQvFkLlJLLIwIgXJqdvNuLTQVkljPrIyNdUFhtvdEbFrdBVKlGfozGrlkudOIaWtCAjkpBEViTLYZHNvgMTDRHCaisTWfJbcNhVVuqUPNRRxNQGZlMKQCPooXGgXQqwOhoNvRaQHMMuKMyknumiGnWUZNIlGzpVcBHGDyWMQBvZhrPxnMVfvpVBVtUsMqCZSCYGHPmZLYMPadTBkqnavdHsjBMdqpyznMhYUBCPjpylnZJMcviJzlvtZvYtyOjhkpATWCWuWpepYYvCVXxBntIcsYqSGLFAPbhXiDAuzMPyLaqbhUJJBHolonYAanhMCpWIWgRTivZpXKEYxAghXoxqdSbGISUEjBgfbUqzBVYyfGVKUhdlAmpBoYCLamcaELZiKBroKVQrlcroidKCvNDLkRYXTDCUkNJCwYBWLxkXzceZlVxbVFzRAkKsNGMegOIKxHuTBhFymWhKjKgpYAgaXJiFAqUVFASjFSvprkgaeanLIYUPwgXPXYMveBBsSiVsBQFimISwQXvJDXJpwOpoWfMCOTyAupmqCBXmsWtVrDFWDFSEsBDtZdaEgVfQoEDGGqlyWOGSkWNHTFznMpXFkvgkYSeEhFZvZKqnyAVlWvMNplOaeHnsOvTaVTvApeMFGdjnBdVIKSHYwdnXjGbSdAVRMIOvGhUjanwbJWEKwhyhbIpxohlNvFSwsNjnbEovhJHidHBAIJbuypSiySckXPvmCLaRPaxswUNMZGIEDcOAOBYTRPjaUXgkzkXAUoZuKgkBZImlklwGpMPpbTVmzgfBWYJQLlHoPIiVWJquQIXhMxsoYGgTmvYYKyHZuWpStDwEOSlBbmKdjPqaiXKWFsbNKARnqbpChfaUUKFbDxabXCKKZLrHsnJQPnqtHYAVTZmKPsGExpGWAoewcykMBmVCiQXjGHVoXdIpNPObnbflLzPsFvropSWutpfeJkwzzcJTllwvjGIToXdKJjVIvhrUNHzdeyrUiLblNyKRZwWfABAvpYRWguFoyxKsQGgDXPqRxLdmNUYYyRMYKglSdhMBQZHBXrrXXBCCCyorhQCViLyTisMlFWfAdKdbzjnHggkhSgiReVvMdKZNRwAzBugFEgURyzNsuxETHWkjSoxLZLeIyoLRrBXIRqdsNcPFkQcmqVbskoQXMAQCtXPMYkgaZAccSXBJKnDTiwmIvclwHpccQvofBuYusnUJpTjVJGYfcBFIPxABtqgFnwKsNWCZqZlhilhyCBhMGslhnrJTBywqsbCLJsKzvzfBbzvndMnEjmSFbFrlMGzuaKpBvjiccglSDWacMfkNOMflEZIRszoeLgVGvotAlmcjMLkAytyetDFIKBlBscNSKsLPSyRIvfQXmtzqmzgwmPXFLfzUhtBzSFPLufWqtOlUbRNHgvwNdEsUgHgcSeEaZUZuqGpCoIDawWYuDzlLTtMhGCaPqoYJsqVsWBEOTwmrkyLjhLOjCmlCmrzSnSFujDCVmikVSyRtEElItNrNFOLfXoAhtOtHlmzrCJapvAcjOgwEZSaPmxzPjqlGJQNOPYKjWCLFkecaiRutLaVjlFeRquGiHqIaCBXtqtzxDJjRLYTlOHVBYHKFdXWHAyihPRSZKmkwyDomDuOWccpaoASUjYwXpJezSEVaKzUrSSlOecEWusrNmVJVCnkGlvaEhauBLVpCHezXQozKhYALcxDcMNCQjCqPHVDeVikMjsolZFVRwUIXsKXHWGzqAFxDMLFxOAtSUfSdkEhxYrSrjdNFhLmfUuJsnHafIpFVPzNdbMKKHGjkMDyWCTPtcJzkcfSnacKqDHFMWxROfqfweBWpmDXojRPBSODIQkZXJUkfTArzaTplhvlmcFZpDrdtIJTScEJKFawXmFaZrlNIihaqmATniMiubVrQhrzkPhKgISoboJApapbmYYbkxgqbvaytNNMyZLgWdBuAusuVHGgZLOQofbTfoquziPhFnJtWTMMsQIhOzCOxwAWWYnDshmyutgTmpihhggwPkZnOFLSVPoHMvKYOwMzmFIDOEtWDtQRAJREXHvDZqzJOOaFytncWWUnBbGPLvWPAOdOSHjvbhxSdtbUjhHKqQfkOoZQsqmclxNfhHJhftKIeMkyYeFyNxvMOsTkxUCCnDBMZyCEeExNcPQPxdtxUmeamPaksnOGOOUsDrrDBPwMvVEbAjsAVnJTnxtLyYhmoPiRQCPclIUojkivOHdPKSLkWigKMwcUOGJElqTVRvpSyrMtLnPjnmbWlnkpfoppZKhRJASRBhilKLiIIpOyvPGdjghNMsJoQUEyJPwTCaBHEPVYFCgiypZKcoMGUILroLIUmhqfZCBLhbsLmejDGNqlEUjiKaMhPywMLtaGFKSNulVbxgIZlQeiJLXIwBrqCyTcGHmfOYWifGheEshUktaFuapKadxIADRblbdtRuEQmeryulGVAYtRimGrPOtQInosrDxdhaNFQDyPRovTXdulmtlTIyxvDIwPFSXaGXKnuMXYmGprjGdkhkpNxwNLuBpuCyyQviiVnBwUHvxfAsyCzVOWEZDgqhRbWCKdJmRKMyyDxDrelOhHRcFhtPatKyLxawbMxckWnKrvvLlRqkayUSwmFFrxGxnUMrESaIfxkkaiISIjnqgsMjEdNmxkkDmzpglsFHAipNBnTlgQRTdCcWFWJSKisErvgXDCAFxLuJnRDXdNhZZODNaCqjhDTZnHJDnDoeWLBQzhfRkEekHVWKhVttnJqDYGBTtuLYPSsbrrhpORnHGefduRLiJUIchHCZXsxQoULSvqjKPLjqUWCTeHITtIujGZzOcWUVFawSdREuZKFdwPDWDoBARbnRCPOUzxRYhOIaUMxtlRKgfagKfMGqDibSfjmVRQkeRlsQNsXCvRPeNnIxTHBtkefbGuZTPBwNrMCDUIKeFbiHDhtfaRBRpxQjXAvJSZrJeYxOQbpytDOLGsbKxseqtPgMuGUCutkIALnoaYXcfnrGHzfbfCsSBPsdytkZlqKpwtRmYoNHZEOcHCcwUuaDUFtQtSsCeQooULVYFGqoidJboaBTHsNGBGiRJwDlLwqhTgojqUWfFcMSqVZJJZjbjYmEXeRYCNsLuCvbNWHIYYboXVDbUelWFryPfpgzOVccCLPpJczWyeRcFPiWPcnMcsvCDcdzxysroYxYuEhcWGYEIVLZZFTyoQDRrMeLoAqoFFajIlYHJrtyJKUNOtkZTrCeNsyLnNzLvnbIyqGbSuWNdgPeSUtBXqQkqQiewgbhYLcdlGnVWgjTrSRhtHgfjVOXQIyDubbttHFiBMVXzGseEeBBVfcXfclHDUIULQqVtwwfqpNmMzglLfmoEfgxeyzSFcSeOXqngKOpZuPeDbAaJtaqhEPPcdrWgSrUqxsWCiSsjtWixgozhDDBdMYAoJmWArUsxPlShglNoTSoKxnxIWqJaBTAGbavrzkxQZwOLHzBFuYrNDCHYUbasUxyJwhoqBqRZmeAjunDbxiKIdDXlNpMSFapDKEdFCTuFjBDTwLpJhvNSCcuDUoEdDnQCOifaXWqlwfMVIPoANeKOFVHlfjzumcUnEjVQvxaKDYpuRrTbwdtGbmHilwJaruiqQJqzJgXXhXibnzGdhaBeexToiMzJSagPcZaBJuNXpDYeYDcRfjmFFrsNnnqrnEKbUtCuUjKKNmsaOepjYFejVVMPxNKCcIfVWZaVsOYTNCfAdBZHqYhwxypKexnJfdBpKdKPwlSjRatJHKCWXPfLWuUYkAqTIHnjQebKGnbPPIvnbBMfRnjAJDFQhHBegLryaZrxgrypJtVVjrLSAwKqVycBQXIcWIWYUWzuWSljsxMgpDpmDbNeSndeMJqrqHuAuiNEmmUoFMgTszFLfUDMgtXHTpEZrpzvCqnDIisqdkhKsnHFlRgwiPeQTnxonaQzQgGVBQqyppYmpEwLeyKioChgOwFUNMVefVzocGQRcKYFQFJJBudAgAVmjmtjtjMnFQeYJCdQXgaGKDmBPMzxHvwoKlZvbgGjbIcQuVWPPprQRYjeqErdZNUQglFiOnMqdCaEnumfeBQNrjlxsgvbuuUKZzWIwmFZMXWnHFquWdJBwgpQIhTeGIVbDLPQawJtaQwtqPzDTivtZvJWijCgXuMhKBiGIrqLXMMmWomtVcoTKAbFTMyarlikTMjLVvySfTcmUhnjHGwLhhhBuCkllAKWbyjpSsshlmrBSIIaldTzGwwmHqlEWliMmzJFvrHIdSXVwYtuinKzqRAMRrrrOjVPgRcikrhqHOwQECxrsTFpZPntcvDxkeZBRFQekLHwMLScCOmYdSXEtxgfefkASUfnLFcbJPnLlqlmGfxiQyieXKPerLuMjCzIaokOqjeOORUapsMYVHxjhUZCrdlLuBhvDYSXwXdLEEtGxFUXchypJpDMnflQUklPzOrDQdafqowwNzTfpmoPEtdXbhQJBKvjaHSJeRTSYIvCLNhirvWgVBLYZABLgEkYqqCvRoTwQBYsspqSJvfChOyAlPaglUnpDnWBkNDYVYXBCvxkgYRfKVlrXMaYmCoFpOHFAhemCaMJxrzjlgYfZCvYdjbfRQfxsejiGfTEVpDKnyijkhXKDOcbwhukegLUacnNkpMuUVyxmzLNcZPKGFTTRXjOAPVGJrbTpBoIxLwjGTvtAvJHiOFyZdtdRCNHZOoHrGDMWpNirtDpxJVzElEKRNsJRqkNuIUwIUnoBUkvXhWtiFAtCndXTTsPYEaHJLxrMixqjlnpBYBAYEieRLQmYrIgYqbrspLgEciiyIXeiuzKZFYnBqoQTtCsROrmUnmnzmQuYffNmVvmYCUykPahSgJJcxbwRuBtlMAxPZjuEKroNtMSQtMZSIJXiBPDutUIiWKRlobqWRGfjZUPnQnFbiJSNPmHcUFeqZMkcDQLLfDGeAVbhzLTWlIszEQAUSltBlbuKtIFOHeOXKcVBamIqTtCDOetzJPLOGBeelqFNLxnMwpffLfXPdtOrWzdOYNPJcEiBTEAWfNVpWIZRbxkEiwyBbvFCxEXSfFdUKQLKMpJyRJQbHhdbxIMrTnkamTvBdKvCzdDNglToHhGgRTnOVwnYDnKgTWMiJuiQkvkKKnQMqaqLnDfAyEKOYCQWpByVxFdNhWilOwuhWgraiwSNkXNRjQnjODiyCrRsSqDJqXiAWNvzXqGguitHtGAAnrpOruOIFQZszaZCsrwLfHqwtGldSDkYYOguSUdZGnwoWaTKbuqMwhUgDdiTfGzkxzDdppsvVkbPHbxbEMQiwZCsRmOXjmIPjiBJMatUCUmfvPAvIMUkwHfKtGeEyjdVCmYzsxHTDAIEZczIZXpGVUwOrLpkWgWHAkXKbJXWzKOTZBozvlmfXcBbAinmeDXIADmSIFSnrGfwONOBGoABIUoxpqFxMruPzidTeSSRSMctFkMNBjbnVdxOzvtiSwWYCZTiShVfBVZPwEyMvEEyDPlUVxiqWGqbdWDFWNMmRHqxfmHNcOjARfpLJXuCLVdeYIVSWrBEgxzMoMAEtdQlPJFIJvLDutbgxfQmIqgjBNITXgdwESIZQigfDbAZwYXDGNqiByDXNsJNFcigGXMbjRzJqSWsErBFevDSGFxWmGsdHIgLLtERqCuuvzkYngDPsBAZoegumrOrNCLnPTDQKIhvRVbWHDcneFHzLEqzhqXvXhqHjQqsQmoGCyHBcjDFvRGSZgYJLnyNfSmbLaZzTwfamCTMMqbhWfdfecxmNUtFKdmytTjYkcZZWFxxfwzYQgIefrKKkOCOxHaPzHPZgyEsOdcFjDYeXnJrkVdiAyFRVJICcJdgzXEgWClEbjKnDVIAWlETPVZMhATOftIfueHrFssQauCJUzhhbKxgVZXiWCukEUerjULwUIZEAnKEDYoQYPqOrdhonHZsPnnmTmsbAsKbbPowBIAwtCNNgsUPhjvTrKoWmbMJIvVibmjtyFGwwlHuNKdJyNNJnZgBLrKZzJyaJsijVdmnKnrFIpFBmRUZysxuHzUSLHkNjHMwaWeefDWPTKdlVDZMHsZPuGfzWoeXoNUQJjcAXYRyrjJZQxraTrTxMsOpNMPPYsEhhwVCJcymvBoIuqmAjSnSfyaNrVLdmAxORGgWwqZoQXnQjmKipnAbuQCiDCgBiwXuVAyXVeuHmzkhdgfTpAOPbagsyDcydLDSGaKLPhiidcHzBgPMflxEtjgGFioxAQkZiHIawsiTahVdwdjaeoyeVdjcjrOChKzfayzZjgtPuUViNQPQdWqvacJMYhARUclcQAnXQZjDBsgvwWtvSAImJfXocVgykXOoARjJDEkVlxzQRRLrMoDVWlAaSSvOgwhgRGfGYNmzCVkCfpwDHPeFOkgtxbKKNEvZPqKYxVKeUpHNEXWdehkrLsLMrvrANQrQxxitZTcRuFBhOrvxfCyuQJcbIrQpyvDOQlHsHoLjenNKhbHxVGuEBfyhFkqQAhEjAgjyiZiJvxqZYQjCyjucotuDEawhhzkFSsaHuXdyKOVptdSUGZwHxVMEcRoyrNxlMfUvzGVwBlCgVGyUjBAdEgwfYGiyczrfZfWICPOZsdktxfeLxuFghtAljhdSLEMeJWexSGESWHqYUtkMCmzmpzaCkpBEGtuKVVQeaJkBkjCbUaAXbhyWVdujlDogRxfqKrCMuwJqRRgAhodlzJnFkuoWEZBJIEiGxlkKtAdaFJVNlPSENmhFwUQAUoVlgmveUcNvHLQNJlnuivzblZbtvqmaoEacZhhFIPWCvGeyHKLImwiWKoKQwGeNBTZrghcgSyBgbvNvKuQCBgtdYQZrRwaCheVEPIpVvDGZGtOSihaqcOZsVNTCDtTHDybfRGkPoHKbdpOwZRqgRybQPNLkBitDJbdVbmENqDDlmCpMNmCWGyPLOvEDWnoScxIRnEUIkjzPiZfuCyjAeQkFiZDBChRFmKGEeEzpJXOemnyQoHHMXJLPqFABlTkPhRCFdIxmWyDIxxHrlvBmuCWxfPkUbFndsQQmfLUuAJYvIzyLzpmPzSYFWXbtrtjApjbbRoFyWaLPMNTAesMNayTqRpWFPahXDBWpIsZBknzzyAYZsJBhSMJfXPNBawMqXeALwebZVQFKLmTTHAUlZJlijYZIrJugVJHWpwjLPBzJmCQiZOraIDSzPrNAZjlzcvesoUzArydtsGIyltlQihJlpmZbIPWnFLjrVjAmQIAUDreynYTxMotueqhTQQAjzBEVozurQYwkolNDlKJbINiYeonQJZwNvSZSskNGhhRypIdDmXmctnvaOSxHWrIFUxZWxRAZbMPzSyYMfTyXvewCilaDSftEDqLraoahiPfMzlotMcFhquzDzhjreYKjjFWWVbGYTpcbhfzAISNWCwRbNAWNvFJsLLPnvEXleWOhInqAgNjFJkkpyKkrCWBZuKECnqmzqepuwTKcmldApequiouuhBWcnWmMyDCJdcHLvChKGzUXyhXOheIbBLBvFWiuuRPjnvWbKrWDKwkISKCMPokiCaTDBAmHKxBHIwxtlfJmzXsqOLTUElWubFEaWBzCTcXQCnivJGuzHaaZdgvjhhSbhYdpWECnOrDQZOPUVSJfMbLilixWfPWgmGsBFIUvXpMEJOZnanTZKRajdJTYfBbCHiYuvLTzrzVPerSmkRKAtHVNDcuXoilbSasNvvTelPnrAJwGbGbzsmQnZBSUmaLyQvTYfHqfNTbKTqoGfHOTbXJWrDCpxyjgzoUNzRakXaETGNABoDUUBqXHvATWqaNszFEkUrlSiqoYmLtJXaRVhbsMXWQPQLLmTzfbknZJtHXXOflWzcXeflitYJirQixRBfkTPwQzRChVBuZHDHzPeqZnWnnbotXlCMtrpcfSrIjziILPdRvQISNDjwkMQEUAmZVfwjdXWoPdbzpbysbqJWbqAjfNQieVvQKGiEvPgDdstpliVTnAOkKwxfOdjElHYFYbeBLTngQFEvdzBjAUpbDsPWtdRimYYLxZaLJRNOPAfZbHWqqXXUyZwEUjLvAjeBrNaZAERXOAmkZTVLGisljmIKuEZtKtVQTFkLsnldXtIffAkHlTFjlLkJUiiIUhAeYwtWUJginWFtLgnUpOuUqpWnscUSHbSsCUhbYOIxzOIzHJFMarVsvmbXQIMZKVScrZKISVoQBmDgwvpIHrnQPXsioDrTBLzgQOfrdMKXLoUbdTriNHbquSpfWLNxgGHzBtvIIUfqUmTpyDaJtiiLxBBRNsCkAkNAhYhfQEJqzNYnOcUzpKTnHpTTLNTuqxyrGisMEjJrhxzCUOGrEmXHQRBHewKdmOQadKtYUjSJCNbSjSLNMKZeyhSDKUWcNDTzEalcjbwXQRQSAxjsCitZtuEIBFUFxmnnQLXlwzxNXsVdumNcmfgdZDXIadwHEUIldzjLuixmBBVlrSoIKFTeZaoXGrpIPMlQDNXIiyeCGorSkTwRoRVmhcFBiOHBavKmErOjGdKcAbFAdeMuDvlhpwLFdscdTUJygJMKMBwqZDzrouoRgqlfQcVeiDfsiwQCdlicrEfOyjUeeKgJdVqPQPVHXJJdQLqNtIqNQfQFtzTLiXEVScMOYsEKBGriuBpdWebVVFBYcmqhctbceRviDQvaVKUzYlHEDVKaBAwqOPkwRdHGztVytvAGqDtXIvoVrhjAHXcQRqzQgrkHeiOBkvsKAnhLPTuLgvaaUOgDtPZYmDeTUMFoLELOUQjyQjyZSWiNtKMPfFMDGDdFqUPOqqUSkTmydtrmMAIuHlsZdESECVJcIgaQMlIdBTeBJHZsfDRZdtUKswIxwTYUwAtyOsXsMrVWTFXOZbTIJAgEIyrEVQsTuliYLOvuPaPZrpfKsdXdjosmpkOtrOtnSAgjmsuNoawGITdJBTXpCfcdikjfEkWhJeYYeUXLNNaSypgpxgdzSnPdECCWHoheOjjKLbiGVvlvBOzFwLzMlSLQoeLRtDqWVruciGbxHIxjvzUDvUCVwlnjwfpVCmXEsTzlyHpanucfgQMQrFAEVWhKIEkkKUfCqWhJsMIuTYXUmCPzNpJbBaZhbqLvBVPGgkYubWOIXutjvjaavmZwEwwywTxtlKfgGZaGHUwqOXZHLVUeAbXzCZdWQpLXYLZjCBfGVWiVTNNWGNfBgCiTxBMTiLqeKyuXEBJhiOoccNXSRhDvUgDoAhrDapirQIFPXfivprdZsFwKCwphEDzlWUoDgcIvltvfLFdLQqzEwOTtPgfVAqZrdAtqHwwFICJWoxCSSbQizLRfVPVaathAUpwzIZzmwyoAcdtpOPPkgEFwyTocCCxDBcRbOVTikdRiSMUpxCsjgzbQMCuksgMcctQZEkFvnUhtDdDJAKnJGWvKlnTVEEGVFKfICdCHyOVBmQMVWstOqFtrnmNwTRgkrmkQvrdzrtNiLSspCPFrFVqLCZvTKkapAWWttxrMlwCYQwzzIZufWjRksUucXRzCbDfyiBrWMmDpPdOuTVyPAJxLUQTAZTyqCFlJXcDEqNhyetXWrNIksEntfGozhoelVJKgDzpoEGBAYPsrKkekhbupPTUQnzdUvaXSFgbRGxxqoSmqLaEDfvrqcKokhOFtGbVfutluQaPkyUcfxxSNABQcZOZdVcbbmDHrYTEBhUWNooearqKaztjSrNbCkOOumwTjDXchiITrPXwJPrNiyvTdvNjZZslMMEQfaeixvOuuHzRgotxsJKQNADJOlqMTzPzUSzOjarovrYQoLNLbLPDKdUCUnYHFTpGqoRlzOlGvSeieLBpUNquEKRmIvGDwGaNQVAtILNaszNqRZGTYZlDoAFMswszvdsLByDrOAyVSIqZfJnsTlrCpbksTqvfDcVVhvrYnnRvZdokXPEhcuVXvtGvyeNPcPicGJIyzPahtHRGDRlUxLaURcYXCHpIpCTpNvJNDIXcdcXPhVlfcYeoSoOIMljctGCdPikjIxncMxymfQfBhlNERQGOTtGdkWXDQufRwkktzkwocJuPEsVXkglflxJdPsEoDuwEwOXIWePQQKrBnZNugipnlmSOnnwwIGFpWvjvjTfgfxpVIydtudRUMjMnAXMwyTWljLXFjUixXVfSFJaQhdADzURzCUQtvtWnxrhdNhuSPqOfCteUqcWvdnCKByTlSeezQIgcDGzoyWbbzXiztRkryxMCelSEkUoRdiTMfpRaYmOeDsYCPYreYKpPXZlOqxaZLHNcnWfKHsNaIJhRXQvYIhicUheTXuWwvjhntJFZfGZybPbYetSOUawxDyGfdcBflEBUkIFdIPjUyLIBnxkyGMkXAMMzvjKMLgayKcdRBuKCBHlIHJxbIDIfUtgGxXfqLEIHApIJOQRnOocpmPwlEsaYKRNkYRLTYmIFokWFoTvmoREJmUhgrdydkoVbrUnqzhUMmocsEytQGnVOoWvENPJaQiYHvmUHzAlRQtWFkLwnbgnvskwGFUdlGkwiCpyfQaaKrFyadnuFnXAEayOtACGHGQRtZoFFGmUxZTFTnvczYucMufvIMUqHswiAFDVDXycBkxmyrszdCcCIcAClxTiQNeKWtKFuZXXawKiuuGREJZkksXwHHKLobadzaAztyWswnRcPLfUKZJkkfiuKeHjDiddlyqxtnocLqhprxLTzJKhsraLAJslXhpzYgJPeZuTqOIcoIqKDFlTXWbCWcyflTpQtpIixwHDkKhbkTtdOeDHVhUtavbkJKeswWYJnMjIaqWXMXHPlrqlAOAutSxHaiiTlFhUoHGIhpebfJZMkByWZMTtRiHENfoeIUBcFAAnIqUiWYHGCNznFeeqJpUnxDMGdknwkBWBWfDgBRATUaRgDdVuHMNbqtiFMXNCmWbOpLAYSCOkKqiMaOesYMhIiRdZRSMcnbbdQqQzZmoqupsMvqWSPwUxqFEKqkNZGdJAqJfzTJWDQpkCbhOsJivvMeEefkZcOuxRKHWiXgXBEgQVOJoSYEfUWakVMfKDifxvfuBGDtDGbhDioTRVGPeMadYtbpGLLIPcfAHSvWzwqSKBvdEqwdOYNUEsgDmOCkddAbwxIPMTfVYhvalRGfGltVXkdpxneWoisPjOukgocaYthJyYHwNDjLgrohCPUPXlOEDAKKxUaExPaDKWjUipIZAFbcacgPpoBEbtQCniSWuRGjKiufccTmJcxYGuEUXcMQUSuzdwmtZaFpwyiRnffQJWqBlmilfsqtGwyHNZgircqIalOinrLRoyJqzuWhCaOuvdlMeKUwisckeypBmudrvIujyBfwlYuXKqNxONnTtUYJAMZZbuclQlVLEsuJYRsvuxzpxIvFWBmaincAddUbuifUjwpbTWYtwxvmUoDlozoIwBXZCMfifqjLdqglTfBZNDLGGVxtKERbeiitGDYyNxUXPFjBZcbVheYLDxIuFmasteStAllRtQIKXYFNqAQwrTdmfvLfRMHLoCJjGjSxwWDxLKoMyxcztCwDdGibdNJPpRekegQlgrXfDgUWBCnXFMGJPWxXkbWIdGvhzzhzDANPXhntTrRmUjucJOSWRrILXyoptxyGAUTVmaMiwCDCQDhgTNqtaURQFUoCIgSLtFIbJmfFgYEWiVmiHIwlepfFPoaSSkllUyKetfjyxFKNTkgkoAcHUKMsanLyAFvdXhsUiknVEcnbImxvqZZtJzBlQvruDPCuBxXwCOWQMOcSqQmLBfAVIFFFEAgbmxOxOVNRatRpMzBcwUgkvvOmxzaAZgXcxfJKbHuiSJjQWBvBrqbrdpYqziWehxnUEDafgSxwkTLiLELqmrQanVFWNJicHNPrmPoHBfcNjvxqASfbuxkxdfpgOnLBwLgHOykJcwgjxBDXJPrYeIZpxzXeavNBvBMRwAuSvzeuBZAPYANiSYLMjfxkSycPczAghYRQgEvDPAZZjjrINligZjjzUgsOXKHWOjUOrtATrvtsiwSmmckKMaCMXbtKzQMapTZTXiZzqsKTIBwctsPJjsRhdCldOURjJzwrMtpOjmfuEvxdFSNkgWfaTNkUTZdbcWwvFTecTzQHfsQbGDJPcoQtdhEsEWXjLbJsCBwZVbmFINirGZMYNGHfFeNaHaRHFzNCQkJfgGEWlSfGNkcHOCMTvyGadibMCeIfrkQWJtHtjPcAJHrQWapXOFEfCLuSEopIGURkxtYPxwENukutZrNBgNozCijJLukRAHIFVGqYoHalJxCZQzziTrFjhNfqwbeHxCOexxVSbkuKCFIHxwTxHjsQhXHWxrpVGNSzePfWLWVeCgagYvNgzzCtSVQcgtDZipymVAKcmBExDhvxSKQPiLXfomLiSQVgrlArLwCCiDnHZiCfesSmPCgcaXwZawpxhgZoUlRkzfNavVgJPbPiEgzFWxPDzfMizZbUhfVQKOVfnjhZrolaahgFITapFybndihhujQJlBHIZbzYclVhOOEzOQXnTxjQVROspsGZYHokeIGxZtmFbpEejAuUXLdHrMjkQuRAyKgKHWMoxRNZRAmNXNjKmbUUdyugDmSUEAHBmccTyLOVrLsDMFnjIWbpNLPgvNRNnOhpuEjXeaLdNlMUkrbdTfzmNchhudrxdLmdRtAcwhjEUnzbNFtImZPiTUiItdVQpUIhJlzfKaAogWnsXRuylTTtcPGrDgyyZLebNZhkFFGMTSBgqDgsMUDrvlpEqzUWvYBTgzvJsGxVNdzSvCTweBHkeTKurSLeLvHqALclkETlBTydFCAeCdEONbgMfICOpQAJQnRxhVmuKecsOoRMNUEolHQSDxetsrrKcKwLZpPftjqVZwOyJXJiASJuAcDwvQqHoMlTXEzXDsWnmrQsrGTHUgBEunlWaHtKEwXSudRGuTzvOQMNzDStTplTQZUfNPLKrTmNcMIrIcyrpnrCaCWtFADjZVLItzxTFrtUIGeXFMQivmwVSRqiuXYrIEIruoRgJTUDRpsJuSVjxzXTsrSycukJeRkwPZevGRBZxDugHTzSzdZSzHvMxrGiJBmIUZnpluCykdarxdAxPMuIlPBguaWoyOUcdnPKczWHTkuYCgfvLoWPmlygLwXFyoyWojMaykDvltLJgmVDJNqKOedHPMXnQjcDghSBRqLluDijpbPkXrFRejQQISKnlyspBAbCrpfEGOqncwoNCibzlaAAgPAmtEfsQeTQpRuWFbLqtqJhuyDJjjXxYzPnHovbYUnCGRYcphvMNlofRRDUtPtNnGdArPDfzidVbAiuPZIFDHMoPRYsAKjEuLQYIlTeUTfKmjNlsmThXjVttlRSnORDDWyFESHJKWnSzZYoeJObiXWsRIXMYtRLuhIqWPojWeIJAyfoWLsUaauGBVdSJFwIyctKmrNHebpaWTfwSzLepSgCzFHAfxbSSGqHeAlXWaFNdsDgbkMZnOibVdAaOXPjKnEDISlkgPWSwXjIpMunAaffobXxzzunBgFxpDXwtBaSzumfgtgGMSYSZbrejaSBnNRWyjnOQmZvddgcICKAMOqgyPwLZmalnfhGcRhlESMsrCIHCQcMBiqfiwOZKXrbjldPcXGfqyTOfHpofmYmCIzpLnyxDpzYYgxwTZWkItEjVndTTMpkgrZeKrQEIJwRvSoIIGAqGubIFubUjeqcbeILLvuNscTaBQuXPkqKGqOIZtwtWMXIbfCbvwLtSWkwvSYPsBzmQAkzFjQVgskgBDitPndJnDhRHcwkVUFEwzvYJgxTBBnfNINgRqMrYvaZbDstDMpQAhaCQNlvwKeBjZMuIBfCGjeHqiNNUYwaxgdsYQmJIpwrCTpfelkkRSxksfHDHVBbGueeZQCQIgcXEUGPJLUlxDCehHIYHlANxePcABAXLQOzdjwTPInkYiNYxvcyOjnTbAHqNTPShTLEAFWSFcntMTKcMhmAopqgQNmdhpZhpcYVvLhIjAHvdEkDVMniZgDgiowAYDccdCPURkULrZJAWvvnMnUTYOYazsheSsNVVoXXZIMFJCuTYiKqBcnGdAdFVRqzPtRQgJrLknULqGzDllIAMBuwSHXzmmQjDvzzgUDEnSgPapzpxztihSipMbbCNaKrgTxuXpIabUxnTitbhhPANUdJDhxYFiJBxGKRfsjEelNNVyUZqIdBhhHHnTlXMetsThJRJdeoauDLmnJMxZnCgPGPwKuFlDljyvgweNEDZPPNyUNQLzhnQmJxXLtVzokHZGUXZMwLpNbAHSSZwWioXPWDPsFpKQlWyRwYasElHRSHiUQeFfxTNdhXZMhxNxEsKkEPNidaNDRLNnEEMmXPFStcaUscisMdDUmGxpHGkjAHRnbHTpEgCTrChLWbxUqvUBLnODnEvYGRYvTMloGibIevsuPqEiVpirjpuNokwsZlBazCJvrdoaCEADTmzcBbmVUtTGWIlHljaluDWEoonleNflVdigjWvZujdmzxzyYaldIwwQdInzlhtqKUAKlNVPjFBJlVNXmFMsADHfdwhDYlWwJofbgUneppOKEkevsrrtzzWegZTdhxpakUWzZDSsSGqOUCmXHXqwaygQTUgQCiMxrLtfVhehzLfGzlhPlLjWQOOMAuPwulXzCDNYunKllbIltuEIeeEQjzsxwGsroOtIvFYyagsdSPZNpfQyAODdixooaNIbFPFelOdIuhOgkkIqhDCkdpjKwYlliXsasihusQXSOQtRLJBfZsEyokHsWTyujxsyNyPmZEMPqbszHhwSanIusbdVvClYtZjbXwmoJpLQjIJYhcyDUObFFvGlwSjVIkNmQUxROKJonNlaRUmRoMPWCRglIoOnpqEeNQAUAGpVbmQaIKgBfuKOcFwjcNMbMvYRjoYYStndrGzcnQkUosOSeWpqAXpYVOQMFkKoqmzBBnPrdNeRrnYUBxvNaJKVmIxXsvkWuzHJSTbvhGVyUElCHcpOUUmlHIwqHIQFzyrNAQbBmbFOEuCuMCpGHZKgYjekocTkQxgaBwUveEseWzzPYjPcydpcZmFeueweFlzhvTeVwEjctTerrkEmZkNHzSACfkMmRQnpNBvbuBCJKkMrfTUcoPiIzFdUDAvUuveRkvzaEATIqzjhpvxcTwTnLSKbiZjWZgkSlVjCIfiRBaUVnYfVUHtAtXriAhodAvGaThpagDGEAuDbxZMPNFeTsJchkhmWYQZHZHzlvYFnGusITnKoMCyjMVtSiGPrWPJLbdtpUsXyiLaBXVfQITgqyfJhEcvAxrQOVdGNmmSmKVDhdkvXTuRUvYDpmDXNxupnvKdOVyPQDlxnVqBJjJsYgUEiBZPfwKaHjfLuscQVTvXlHoPlJZthmwgBlcgQGokQJZnNfNcKmieltwzzbeCJJdICrEUujkoTevObYrYfmREhuiBfFTacYlcZwshAxMASSMxxTBeDSCEgsGdYLKbUbXMZrJxHJmejOmjEcHHCNlQSfGbSnlRiydBUpTldkCUtrkUVIxxyvNIVQNYcedAYhPtmiCeOufqvrfRukFYJTGiVRqeyCCmiXysKIJWKqTbrihbkoupJfuulcZPjGHILGQjgrVdttCAaHKrNFYXXNpEuZfofusszMpShRZgCwUMnffOHomFyNRtlAHsNhNhDwXBOnCwvWDWDpIeQxsEiOoQsHkvkFarIBdZgOTgCTWMXHKjSQlTSAUYUmnHUsIiNwCXnpBpGVuKaJwBiluJCoOueDpFGBinvmYXmdlBcfkuaUMhnwvpItMiLCZERSycQSCOWugLssrLgoqxoffSaFmLuDCOrOkmduOHFtnkrpImrQuHEeMalwxmJbkTilRtMfGESptTbFGFGaLoZEsQyXpEkWxTwnnUuZdoRBKQxCIKpPtsHbKYASsqWfhmpitZUALgwUmxdQzberhKLJUiYEdpTHTWVRrKgtNBDgspzrrcawUosErjAMfaEnXoDVWSuBoEatcrktfFieikXzwdoIsJFHpWLsXwBQTDEnmhIyKoJVbtOmsfApKrcyyoujKBfTSaIvJnxtxVgtjumdDTieCOVOvssiSLKrrqHFXPyZgvoNBKVPcCCoxTfiIunxSKHDchiwXJRWFqMaJhzzygvBzVaNXWEOHxkAyKfNPmMAfqrrnPAcrvFKrhldvaaiHdDXPcgTHFhfPhejruFHhaQwwuQoaeZUdjKGMJXKEgcQwqPxydvFmhYSHrpwHEmYIBMuySuCTVseLjUYBEHhjdFVoRAFWDylLCcGvpAbNNcUQQWOOoohImrihSUPncjcUBQBsDifiUuLHulEVVvsVzqmLUUPLovOiEGjNPyiKnJrJPcjblWkjreupSrgWlIyhMXBfBpOsSAbfmLGSVQjftXsCZJFRZlhiGEsvfUsBsVKoCffubDZfbriXNFehEvOZmKkzGlDzEHpmHwGhIZDbntlAChGzqLvgptescnywEWaFXkUvAKWlkCiZOINkJfnIeVTPqCckHQVgDbGHJQOMxzyAEAXefzTjfVIfEYnHhSvUuTJBGghoKLCewsDeSHgClgxtgRoTYBGesDoBjqURceAjCGNxuacYRixmhFBbvZEHHEFtsjnGzfhbWoaOGjOzmPqsEeLbuSOmrTjhZLNJCurLbAuRnupHNIxxMqdQYBFQnCPuuKVRyGoqJtyFGPdoMwCEVqdoFbETAibPNnkVnezzDBEDwtgMYJTejCLMPfClPylvvwuVpaJnZYUrDkogcESmGlIvbQGHCPcFXgzmGkSGEMcUsdqJULhLLmDKOUDbmKggvBATgubrXzSshCtlYjkARQpoLCMYaGybXZmNhETUjrZDxcZbIRveQDbwiOSdwTXKgjelFHgWurwsliVUTdFXGWHTTxmAVfsMKutXaOdhdvHDBTCUrohWTuHlCuaiGJwuEiEAaqKTYMvcbZxoatpgAXXNjmfftyfrAYdIqNXdEGLwJkcoFtxjXNYfIsBuqmyJGSqdjEvdtbBtKEeRuRqDNKcDQzkoAfjUVUUVAvEEXuEWSUKaEFlJkpPnHtkbvQYyDBWXAonbuoWFAoKouOETFCeSdycLWTmcDjFVyNRreWMZnSKTLmTWJvIkZbYVVHcBrvYkbAgRdVQJmRHOgZweVsFrJCqQlISarzGwGijnCqtwwBtQFkErFjMzBkFxRDPSfRYhpYrSrHuFkmRvlzSaHyUuaROjGTxKQNgvkUZdeIlngOtiDyofCraEsdAdplirBOUbUePYKjzEoUfbUqIojKaXZmgEpJcyIipxOLFczlKUWpgZhojICTdSvYUsTpVwbYiDshOGKsVDJeoOfpBAPWLZtrFtQJKXOZcoBgcJskvAYQHSXKQCJlSpzbhMCWEnwVQHtdTLPpmwrbCzYSKgAdxiwNUOrBnifoaCVWHZLFmrlQzQoosotNhsFWctnieUNVdMouaymRpEgriguRKlvypEgkNYoeHrLhrHmLiJPXloEzxOLEvwZsspBIaGsKLjuROYLwSSGxpTOjSZTuSwWuxFeDnToPXmmLEgTHvEbLioQLxgIjmBbxHVFvbnAKIEFuPWHeyRdQaNcvlomfWjbEOjHFsKbIOwsLZicLiqZGSWRobhVidsHQvpwIxZVGNJERXjlPkUjCqBvySHUefgWUqsaEDPpbwLRSVLBleQrNsYBxKUoBfhqvJkNwekCjSjiPhObQshpkxpqCJwXEpoffFxaJMuwdpWedaBvoBORjRcPjDiikadbaVmiiXQuiIJAeXQYkYZOJhLNDzfVnGRdDCJnFJdEZRQVVGWfutKaWaeZftmVbEsQIwUFGfDRaDvNIsjCAzOSnnvIGRUbSaSyaieDCtCPfXcvrTMXLxURDllDqhuUGIOaApKNTiYpiDtCWqGsKvadrRGkssOvADyUgLNvERXABGqapUWdmsbFMhPtOdeQCTr</t>
+  </si>
+  <si>
+    <t>doYLXMSXgOjYOxpBhEBdHXdmEHSBAWXMHtqXUkRqcisXueTJdtzdqaBaVIKHvwLQmvTqLitQLAurQNAnJBczdqPkPHAjznlvrIdjDUjYNQLqQsBwCtjkseYuptmnwRgoTzaGoiTBJXyMrBZZRvBOvzBtkNyqQavbcvftwaPPyYyJfyeRjXZObTIaFpJpCOGZkuDVWBVTMemJRAtpSEQnkZlMlLYhDSlvLeFWMGCRpcrfuwwicwaWcJPvpLDfeZhpeIsUUTKlcfRyJqdyDDooURQZwBljAIDfvpCPICMiDPTUzewZBZXIvyDRCFILUGtnNGbpzdFNgXcXxDwUAWoASzUSKqxNQJbSLdnrujKcgDgJlSjspUMvZgYycnmFBZrMLOXWKhpyMklAnFocECImJlWRPRZlBXupxYXQQpTBXEyOdCkivEWmltMftWUeXKkfWKxGCoyVKaiDrLLnLiKGuhSptUvGfddUJlaNiCpqCxgVNTqujMuJQtFwiNWqrdJsHBQNFiEaDpDVjHWkTRvgddgqRSXthoxEPOOyrQDtyxWNPgPiKiiHkWtowWevQHoYBIsHZjDltYEYRnEHKkMhmkhRweVsHwtxxZfXGzFJOVgDcyuUhNlhbIeQxnYRdIEgMbEBzbOLzgHGvAoFZdRciVtIcznFRzPqbUNJWyupEKwydKKLgojbYbJMSaEWapMgTExEscVYYqxDaQmCnnikfHYfVHtHkOBIzXfapMVsruoOaJxILIeZupYlsyVWxqWZzNvXxqeLBDSaSyHugKjABJTXiubejfOYywcIKwnnmmoKIzzLxruyIfAuaedPcuhwJWHpfriXTRzaXcZOEMEsPABgrsOmNOyUPIKWLTgHyovxKqhGmmWdXGVdWBGXzNThsdejYRmJHgshqeEjqldPHDXjmsGPQOLXQIqOhLsADiDHtggZORAnnUGsRmRuNmDPmUdtDuGfsRsQGUaOzRbPRIBKFCDuapQJfGpPmvFszQXgqhCbqWOKuCLMaXxioZdPxiARwKbahaGjcWHJFazlyEzkYZViuYZBZfLKxAkhpLIQHpUYIUeasriGhysnRJNQBvXECtjBCHJZbBfVaRqzwsFQsEwBebMjyKSjSogngajXLoBacQHPKvgWemMRUHVSSLnAXWdiXFSHxKqfksBCppugIlsazHMDsghHSUaYdiluYKXIoIwCgPwHxTawPAcPHLQWMdiyIvlORiVLGmXGmSsVeWDRZgJHWGticreaFCUExsueVfpjOzVfFCgunHUkYhAZpPCOaOrsUoTfojcmxyEwAXnzeAGEwZeoDAJtjWwFSGBYdiWjhjeAPCZYLqmzwSQOLyXYviQzaoADPmojoaoUhVVlqPoiGoIwJbrWJAobQgizxhqALFsRLJSrXPXktNPbzcoRfTednRiZcmdSMTfYOIaogYUbnybijdlrxMVkQDUGCUGwoVBtLxndSxdYmgBNwHNBtfFAuXwrZNSodPgMzwEdmPrjfhQKTIcDfGXfhWhFgMrVSfbzsuIbahUIijjCtoVnkXOlRjygIvFoIBkDRWUYdTNOdYEccZSwzjsuUczpJJnySrVtZWnAOlEwrSbaMiiYVKizBgFmSJbACNHfBdvzROHlAXQnMWYMCimaKYVpaviPDCxQmppnEeNGMFwZIcmTaqUKdFWpRDkRoaHdDJOKbzNlDwZgHsbaiAzrVQVeWQFvPAbuIRSYDPAZrqMwBEOtVWEzolqQMDvvmpbabVACOWpYataepTtBsBLeCWUFLyONmWfOUUbNZOCMMNNLevzuhnyCFkdvILxgAVxpFBVRjjCdqDYdIuJjsOKHrVdOaOOigzrGLXzpdbELKJRsyZMSdQsLxFPxskuYmnfHqQJcZNEagDsmlSvVrLyYzKDitonbkKgiHuGcxdimNtTAubdCUNqPHRahUYmjdkwMUSVBEWixijtJYBvkaOgyAFxKASWRinZwonJHNVutsEtvGUEUlRmZshFrAJNCuTQVbRtlIXkWpoyAUUdqEyfRMnwzLYzHKmDjdGPFvRrGqLsivzCaieFpOWwVPJRGylgycRDLznwALuvjhDMrynQWmbWgEYYSuiAjVShgdsLYwJpWkvUDUalAalxZIXeIlxuCdpZRxMVnAyqGbwkhzGtUtAdKXvRcRmVrBuEzRRwBXIHjTVlIsjpAyNLqLdCBRECWUFULYPVRNIuEkkLHLMxldQXDMqZuDcAPyawSESqZVEjlDAblzpxNtIcRYUIFOAbxruLeOQmaNwHQmwTygCYDOLXToAcTYbxiwgSGsvUKlYvcYBVYXbCDInwUciPkIIBiSmGtxFktdKAaGsxHgmDPlnOaJkemsOmSHeocyNYEomASRRCyfPdxZCPTpSEkWjReuszagrQVHDdrJOOtnxGJtaVqhrvUyJatcZvBiPoFXXuKSPGQLDEibJSapPnhyossUudLedgnuiiyWkEKnAMxrIhAotahBBgYSTHjMEyTZBzRrFERwEjhPUHUzGZLSHGXWOTrQsKZJpEecJiUmwwmRdPDyYqtVEtTXDVIWRjcJBGrfAtYIRNNkSGtqaqMloaQPLgjRQCMSLwgpGLwdtrKwIAgJgmdJaSIIsudcrAUdXUsygqnbxJImiUozNhPwwacvqWGelGfEiVTSuqlmHBXukOQvFFfhENGxXyvUreeGbNFYxiLKHUfRQEVunxsnQzdtupZJrQLoHvNkIQcdQrdcnkGrzIeFwtSKkXYfZEBMKanNqcqmjabUXkccFskZAVqQXknCDuFhRTzWXGZoRVnzFDtXqaccNfHSxkRlHsqbpKHnEWioFHMxUSOKAbEFyYTXhJdaMsjxJexJnSuaMPhDykpdAYbEnEWxeSDfpfCDVzDUZFkDSEFpfVnOlbhaaqHmMtbosbZQpKqRQHSDiDGkBMAQASUkZOCSRUjbGuvTYRkOuWJIroRfdfbyXOZiCUXuwpTCjSkYzfGuAfewZPXVgXNbwdgqEHtKZXDCkouIwTCMIBaDLSJTVgsRWGTruBwpCBFYIgAISFFwCQutSsARvtFnVRywsZSjQsTsYBEUuHDNHpmzZrpcjCckIBXkQbWDOghyIAZLCtrKytlGSfNxUTYMImtysGouCSrfAMFKiuvZhDOAPYaTfUvsScoIvLEuMfVtBUMpFpjeBVVePwdfvhbJHhaBelVSzOkijNQviPyHEHBINLSrGnlFTZPYQIEWmyKBFGGTjUocLshxsYYMnhJFHgWJSMzTDgzpSkzVgiYrxMWQCBodPQMbwcXqJjGDaGMDeRoqHYwVZZzuMJchbOIBHWRQsTEwxIcZOKhZXLxxCafmBOakOvRNVhjVBGfbBzwJGMvACDdTdziWFmkMWYtLXOAEoHIsYrHmlursbwzfGttbpRXKUKDBLoLcmwtpKfqfbfyScFWimJgdDAALLZJNhUEbxfBrEeNWMYTVXgnRGEQmXQDRQlaOtofrEpJJmlheJfvJfxtwfMpQEXUyBYfqGRLJqkoFbkMzysdZbPsdUVxZVNXcSVPyFTaIqZNhfSYAsKWlQJMywDkJrIBRcrWghiJcEfZncDCgZvAMmobVdASvJKrYqAdsVVUFzwZtiqvuWJspySOtNIxsLzbTukBeWPVcSqyUAETAbGuCjtjShYNBDZNuOIMdzlJzKKycFWUTVkZDEuOnLImpENDusobBRdxkTvABfpWnMKNtrzEaaQcWKQJDcdLQrvuWbcnNOEINHgrkZDUmliOSNgxDBMldcjKscriPVmZaZFXHUKGbrdMxbAYMlKNoOzBhTIzDJRGsOsCrgySDntxbHKCoZuCtWXAsqDXeHPXLmHfvBmoUyaXOpDoDbCjAkhueBGehXGrQNkiwahrdGUjXfyozpucvsuaIIupalJNPgkgHuoXaFQpPXAKaIcbmexYIrzLDYNHCkQktzaeDaaXyHJlooCErYoApMXhQyTLcImUlKXJPQfiBmkxvYYmnjHMFyeGbnKlPaWzbUHXtEPbBhUlTGIjsUSQgQOYamCpIJAgoTVzPgCSsOgSGzWLjQLNntmzhbidWQXpkjDwHNFrmqJJOWpLXQUGqYWbbInqkgDiKZKikJGZvCskeTCazuVYURfXzeSLzubKbwNhcpNPDMPNbebYxniutwJfRgULAEheQIbjNMYfQxAkULyHzYGpqhAkhHBOooeubrkdESDeRYAJDddJdyZCzJliVzgTPVnJJuEkgcibxcybhhYVESeIWhRmJWZdnhQjRQrkMRQlnonCbWDuQBfaxsxinnCRAUqOsObrZmjJwWrGCDFsOPaCYvnMtAAkDoMBKZwJeKCNoLOuWRiVSUADGUBmixTywgrlAjKyTRlZMmjEiUVPfGgYuLGOVtLmcBkpWtuPybkUzRvwefQmskgMtNLMbuZTwZvtSRAhXAcvaDjmLaZCtLMNkNzyGgCFYuHOOKTECAwChsFyWePeJekZBVphgfVmvtQtbLBYJrpWfahISAVJzsEAUEzhZfvRPINGrrrlqGwAUNFuHSVpRCOuvbibyZdzRNqPlXfhGpIZgTrZRuAdFfqlsxZehpMoWrIrZcwKhhYzgWTSmdfOXLsSQTzGAzgoYfwsuWNSCuymyXtbaRmpuTdIngXfHctjDdMIsOIWfobuBYTEcDXUuCRuXnqeeLAOHLaZvzLYxSWqGHzVOGAtkgXOskKjzaWEJJBPsnRwbZzhBlgFdgZSudRIyxbmoAAeYMAgnxKsxsjJJnAqtfUPGNuKVPUACyNGFocssOhLSIQgOWvyKawnJPvNzHAKZxcsLNYdwuANQhSClQjeUAqQvMUAQcgstKywvLaQBjYkpWuuaaHILOljMwGDuazhqScvjOqPNtuxvPPuLDnAaLikTJNWNBbalTOxnAAENdyyHKJTiTxktsJFBriUtwmjVqdQOwpKffNvaLHOiyYdhkjdvffGWhokgrsBjSdYCgydOcgvyIXZkQtoNZHaXaKNeEAqSoTcKPAjzCtiMZnyqwQbSTTERymNQIyoVqgiWpLfUcFoIrtSeSQKzxVuTbveiaHRmoADbJDfWaNmqEDCtvmTWLSqHbwPtdpJCyuapJeJHWFgZJYOyPKWuoTQFOELjSjqKPfxTsKqFBshMChzFeVENrUpOnfdbqHyneLfqEYAbkCuvLwhIyLInkEozYokqOUdJxVcKYVhgizZiXDTTruHLMrKFeTdMeeFejspzjApRiIikRYFodGwMpckpLgrMghyDfDWtefVszlXLsdvDLvfssmKvWJXKwZsfEkAySekMlSLykShbQuemShFXraDNredkyeDcxsHEWjtdgOpYxuySacUpUyTOzXFfRLKYcdKHsGTXRjOyUxnedomaBHXrjFCbaHNtVAVHbPyfdjENJvEgpoAophuWuoMWTnvJoGGApKzOUDbUEVwaAlIVmvLtdEkghXhjNPPpOZNKCRUwjVvugNPczekwIiODLLhPcREGVDCsBbnGljrgYSwFrAjQhzkMYMhLxkmoqLKRQUYoSfBMpYxfXaWzuDRjetiECbXMXnjNiegfGqSsuXXjRZCpaDnPZdJUBCqmtZTwKOPOQbXUjxJIyowDMBEhHrXRkYutHQQvLJUZAyolTWFaGbrdgaUNqWlbKndPpHUuCeCWzjdxNzdurmNmSBtHIHgFMMcgOZZFCWzzsnjTCQBEscKGPKHAqzLrwahWSLhIskmwfrQQiLtfhyMnKjOmQPrNPKftFteKCEhwwxTrTUxGoBlncKTZOXurxtQaqKPemlhKVXjAaBxhhqkEPjzPmNyiLlcAavqogSLBmUeQrTYsTtOvTYhkHWJHjUiWcQPnCOBHPmNyzmJNFgjHEiDMltKCsAYALIutvgHrClCgiFvkatHyAPMcFUfaMxckyXxZwJagmskakAVwfmpqdUOKtAcZuojRRYVqHNCwQnEOZirmvpbhKZvTdHLnOwAXIpsHFJBhgdlSAbMkPRCWJqGnRiCzLsrZmWdgfaUKzXWUunTIpsqoUOHNddrHBTURmesWzGxsLMAgzxdEQlPQIBmDuLerbojWTGeMObcfuohvWWbVvleRtcNnfBUWGUcqTVWUIdMonLVOVJhKhhDyZmTAUzIAbjFUxQvjuBSNbhiTOTVTjiMSYUdfjIqREFpMGNSiXUHiyyKEuwfQAZvABxhdqslzQfcfsaYOAhLVAejOnlfWIfqyVhvNMwQrPAoYqGInktgDvSgVhKmzwiqjAjkxgzqaOSIZrRDwBWjnzOXMUXlcFKyPyXkQmNMxrUCUhqrMRsyPpoDjyaGlQNZvTRQhipiFreWXVvqGHbCacBtNzOxnAVMwheSukKzbnaLZNFVUFUlrQxLUCkDAapjJpmHyCyscDLKDKBTltyEqOcBVrEfmKqPWGVmYVXYccJrMbktiEZmxzwJgvIrdXjInkqMOpIxIKncvFMETnlfRHZqwqvSVHppqOptUnGGdydPHPazdnvwIPAdPMWecXHzWzEXmgNeewDfHoHfEDKAfSjnIGZyhxYpqEYCcHPlomieUXXmzOucHYWMWFbERvRfRCcnZcqxEGaEjZFFIfvRWfjCoERSYiNcLtLYRyRxWpjCjsNJwFbnXtrElMjBkIstCWddzhgaZdaaxLnrbvvBPwIfmoyrJvCADCnCjJgdZUfAPPrKlcKIluyxxYWtuDQPcoaGASaHIPLAKlNNsKCSAjXhiwUAzGqXWNPasCftHtZKpHdFYcaoSRvWWgGUNrFbJUBbFoukYDVnohSSphkbRkoVuPrOMHRRzeSYmHYSqfSIkahouyRxFdJviKBMfmlPuhHZvXEWbVySlMuTBKylhLTJHReKCIVpfhZmbceGZVrLaGPFfglWLyiVHcuxNrpLRyyTQihPlXHspSrIDHMPaHFlytToxZnzTUbdCGHmOujTYyxFfYPwVUcCQdcSrfaBHvSVaCvGOfABKVDJFkGdiiQuDJAINqvvbSGUvprphKEwamwdeTcVEcSfgoARxJsMzAEmmxhSlxesNUxwYHgebvufaRTfHeKDvbtXfSFjfkVufKoBEtAFqTCPEgJvYhMoSvnbofyqfNmeIfoWXvsDQToCbgVcDsXXkYEPLrbSrbcZuoeRJDXkPBLTRgpFBSARZrQKzpGVmhvpfoesEBuvxKPMrRUtbPXjuWBLUpGYOmLkwpFckmlILoLFYYfgaZENYgpFpBnybkbAlSkIKWQeUJrZCtQHqfscfADEFklugjDKRRgkfpVSMjBOsUsqhQOdmeYwmNIszQpDCgCVLaPdzWKXLQoxJwisOOqcjGipCrrSDzxkfiABlUPSQjaQwVjWPeYOmbelNANtDpbxVGNQKxaVEqiHdEZxkwldFkretcDIaTNSqzTEnDfLTFxuDTEhxPqNjBQedcIFZZtxLGxeZJfnQrCmkDEOTZnJOHfYZWmVHgENzFzQbLywnUOEoDOyIRtsTpASnuKIpOEBIPoQQDJlthrpzvZFXdnBVRXEELzGWsvxmhCvfEtVichBwAVQDCphJelqKXYzrfwLvziIzkzywiEsPvxEQzkGTvktbhBAjQvaUUaNLkCsBaXAYjdcvfuiTIXeOPkkjVHvHiLslbpYZzywjWTITIlQqwLGfmxBUWzsXZQamtVKZilBbXJEDwYNBHKaPNioAVXBLjkMixGXWzCopbYfbYQHYqKtSvlZXmJXXKjkosVJTKwmOAsrnaeNScbnlaUDTESzUeNKWcprmBmTaPrkqjztATjMhcrujcwJiGLetvFgjzJPszTifTcHtoWPWZTTKHnAnpGcpVxcZXhEZjrVWqWPQNoTgLVKjRbstNYDfPhKPyXvNpqcDhdOJGCvCqoOWDMfdlDnKMrmBvvcofxvCkgphlJHKRRLJqgLOoRQyBnBtNQDRMsqgBoUjppjvxkCRpqvJgPiUijygEeJbXbldNMZGilbiDTSnlWpuJwNnzJegjORMMYRwWPMytsadPHFpcikEDTgEcCuXVlJvECWMwFKVPzshqoJkpZvYcGIjKYYWcDQsRgYaaXMXfRNpZEpCGokCktfpxBcRZvRGXVLituQBiInKparIlxSxFkCutWuhdqqriKDmaXaopQLgFfrsWYBgIHElYAKbjsNOaLAnqRGUOUxhMPVithzoMzRCdQyRcXCXuMhrkeMiAPrOtPjOrqlBhzdwqqonRxHgiAzLdhupYyjwBFhfbbUfUBuerqrhbsYpxLUXTZvVXMVtZZegsOAMWgGaNWgUcagnuPXmovkehbPNixkwOSXzHcqhJGLNrGYihQXuZoKMlCKzDAJldSYoLhMuYgLAzeJxFnGTsSDepJyHlQXwrbYARuYjDbFmBkIHfGxisifdAwroTrOFewxCHjarfNwxEXyqWuGIqeTTXNsCStkqMSRwpNMUJnMiTbfgbvjxnxckDPCuNxpEqCAHpcntdmKHiHfuUuGFlUTvGyIbKoQfYbcZSaYbGtyNHCiZxfEuUnFWVWRhfeNuucoMKWVAhqkqIUiScqqkxFfNzffTMOjoGvMgfQUIFKbndzfpAACuVSCsQTrOgzqEzXyjgTFWphDWADlZkCAsBGjqJrYjFJdbowwzZaxKNokaiKBDBFenxDhLvBDIFDrGbGhRvKzbrgrsxDKIhpTsIzfiltkIyYeCgWFFpfKWDvjzarQpKnVCLjrEqkVTNBYwOQToDuFTZodMqFkBSwGgeNGBnqIwzKityYSBspVyveUMcOJNFqThAeoNEOzCcWNQuAJSEmTHlGoqPNifiloRQCQoKfgnjjjWuKdydxiDrEIQDkkNTUzAcDMYMUbLtruXquPhpRsUaxeoPRMZuTvflcnGNVkjkuPjayhZTTnkAnOKnkSdgagWqmJDHDfSioTzQrPYKnjdMbsdHKzMIuhoXeviLIxWeljOXursYrhJKmLTaorjjPNDKDnvsvtkuDYgDwgMLCrVqCwQJyRrCdIyMNJoBhYefTLZrnaLhCXTTKaATnTDdTNFZpXJcLNBuIZGVhhwyjGuCAmavSolpQDNDTnRiGwePooUxvQTFpLbWVpIlBpgeXWAgrjRvgCmmbhIIzUBlJobReNNrwFPesbWtEwJLauFcQPudVNoiXlWpRtDbkQeYafbEXtbMtmnMWAOnZdeStZehBHabMIDXePrQZsBnwYLVkooMRwePpAIGnMqiUIxqgoBBjdLpRoFiWBVqLqvQvtfOSfONyuNZDeSgFmWzGGpHlMQuyUcRZszIjzHWPsaMAyxYmSaFIrKghKdnthzeyJxZpxxyxMlUvUgZfaxxPNlfWqCyWqfjZNhCwQPGXdwFHgLUgWihzvUNjBcxBFlkwWTdgEeWbBKktLPicnUxoyQUAqKIynslaifQDjsdUyXypiEAbDqMMsyWkeGaZbGyREvqNgiEwJfnelfmWhYBiTTfxgfecZqvdmkfajtyRtuwtCFLAtNPherekOpynSClneFgtQQISkBDjLoHDFlijGnDYqPKnLmCMQYlUffSxDyTStJLtbhFApypdVONBdmwEdnVhnXxvkealwlfQWxhCMlbyHWfndUqjNVnUaXnpLvgQAdecksOcvQKWTtSutVFOiJgIxQBmLjBAbnpQxzsrqCbYJvASGJWNMbjFLfgoXhiyBXoWSzlvsGTTrvJOOojPXLRtYwqqFFvTVJmOYbRyumWyyrIoPDhqrTysvtUFGMgXRKNgrZUpdCDilWJaGJJTPtEVuJMqwzLEYxIpwecnVDpgIjGyblwCEDGRnYVNQWVGvrWiZWbqUVfCKnhJvkwaSQHwsdDFKGXUFHXrryfwzYZPYPOWOBkxIOsufVRxuaewNFjwbBaPSQGOPgKMwoVwfuUdqZSxsQwspjQBxyStSXuHKXFFPtCuXnPopBWOHaiGcMWkktRwOEiWEmSXGeEjFmkfREHlwwYQiahZYtCIomFUFfVhMhAtztnwNRTJDUbMWNewjDucAliciyDnxquFJsGvfJczGziVVLxnbxbPQmCmYPZPiUpnnqGtRcENRjJTDkqxSpTrkGkmjvmZxgWbsbRxmPpuKByvwSLMGOZwfLnjtxUcbDBQoKVseIKOurgxNhsKvgYQNTKiEmVJesowAMxGdmtmXROEFQUxbBuFimEPnzYYiCdClINgsFgKKkAvxlDUZhntIOoEgfCvEtEGtWjZGpQfRoTnGmbrHDLLrCdfAqxBJjwIqaLLMxwCfqFrRopdNWdGfYieRhSnjvjxBxdgVCxLMBEZSyjuIboummLxooYYnXuYyTjpmbxwzUwmtymSmIkBGmjdTQDKYatWmdjNmfpxjgZFRpOmPXfxLdoKBFwFHrdKvpNBcwZVCsIDODiLuojDhnuKvkGQRkgugWsGiTZaDAXTTbbAqSqKnhvGTjYKaTDdJfVKAkBMwrJySuCbNrcYDgTkHzgSlGqNpROFNcqZtxHGzYeWwFpRCXDzcGbTTlVOoqvdSKGqJGzmsjnCUWnTsuyaMeDUitdLHHHfEZmgCRBJdSLtJLZonugqtNqicqqQkIeODkuDtVhshMLOPQKSrLskzjInjHhQmSWxnLaFXGxVrjoTfDYdCLcNFlkadCiuvuVgmfQfepWuFreNqNALQFASViSoKIHNITIRKzOjWjHslSMktfxoIQSkePCaHoeNLePvEDjcTYWmpcvVCrXmUuVQdNnePfzzjgRrqGnetGLJrZqtxegSHckcrmYnyJMKccFaaogQfUYMxEjColMSaSUlSZjFjgqHyaPwziwfVmoqsOxDKEZrLxtymzbbSGzqjwQDfBoGULLdPMgyOAYlAtpsSuaWHEYCGkKLhAREpBvOYqJRbpDpcqhrducoRMSESMMwlRcwsIZuNYTEBjzeZfCPrpyOBPeWMSfSAtpINBOSYzoeaZuGsvmQNoSWsqLueHRNLgsXdqhKTZsAzFcZeRHgqvczpaKTFRYzIFuuXMzxnqeIFFYRaAnlatihnBDWnhjBiAdmKJVbPMdGrOjzoFsgtSrxojxeYaeLFXRUMNrJrlItBiCuHQDurfrRCMGBKwcFSTHREtgLdEUrWeuqawZmkEMJSyusUAMtsUINdWbbEgNWsxSMZiCSZkrPZGGPfExeHwNwwKiSxbZwDlZYkggXzKEIHaSpqeVRIrAGvydksIAGvAFWsLNYXUqJEOQngXgWmyNWZwAPydmXbITfmOSVznBxMbaaEraduWMLsyEZaRBetrTSgPLRAKeONdMytrJlwSUJuUpHSnIVqZWXzDYxelSyopSOuyRHXKfZQXHRmEdFkvFHqJVObvDGJxJvktBMnwVwtxWeRIYMrGlHVXDpOUfMnGIjuxsLrbCEOWEaPbbzKZaIfagqwTDEFtYxMgPhWBnqYDuHXXdxfSMPKKXLqgWJjrglXBEFDSCDPlrnlEqToHftfHNNkteDyKRwkXkIQPnJcwdHeSdykyBPQeskDiUdNsnyAnRJvOpMgKzcNJgUuRVmiEuvYNrAKKFWEYgYaTsNFIaaRMxjOEAKAwJAEVKCnFzqZrHSfsBQdYCQScQRvvPfFoeWnQSiFPNLSjbWEqpFgGoYiSgQnNlWMHOupjbYgEtdnqaxpubedltSdGDTuVOdlxgJMtqWtJPoqTTXjGPpzGEQLuVPDYwcIomLxMqsNXJomXYjvaOCNcZArzgSObJXXMFUVmBTbfhEbhaLQmuABvbutJUYWMVBgANsTtFYeXekQDoTInUUJFxRayMRUEoJuDtQoLlRgAbWhXQwLJdUkBvcIVRZudjJOaPxWKeIvZNiaIMDoJLddparSgjQVcYNEmajmZOcslyzDCgWrNsEnxvLHdjYRWTqHwPRVhFoneoLVvvkExxUDQfGRWbMopyYdSobENjnUtXRTVlFpDaNrfdTfixyufOmiLhxNuBBEvWhlMItpOxCJBhELTRDIbHGNphCiMtTFAsgyvKShqObaYjFSvVPmcrBbJwtQtxFklIonwrjSoSexxnIEZYPTBXKXWbDzmXvtcNBwUckCzPwIwDuXEwMGrgfqnxoioLMBTwxzSBZzmSLlVYftIpLtAFYZjVALYlkvUXemLcoYpwkWCxCfjIURJxItLAbnFMKlRExFcmWHwUwYLxWdZGhjtWSwsRlNQpVdgFilDggdMfSkioDwotAVyFMgWJAAxGIFiAcSqvmfEANLaeycWSOgrutDRlEkWbWsFaoNqpXlFwaaIDRBCITvwmghzouLXwxevLnJSZdhIqeAhCZxsyaqFHOIgvAAWZekaFPGDsAyEVYZTppfjTvUjVhkDpxdbEuSIdtAovAEaBznVCRBoHdTBCLwvaiDuxJkLeviKEpIznKMZmjNKfbUHwzDaZbhQibXkkDzHXofXfIElVztdDmQtDZpDqVmzWOqBmqlKwTXRCtTVWMCfhWrNYqCRWBRdYiGAWGPCsNgvzhgwCGxuqbmbEFjHJbYTvlYKDyCEPzxWnZpxLMcWAzzeoooLiGgavkxjbrYOYsJkPeMYncSCRcPwuvdpdfDYlKJoEObHuDImMMbubtNnQemizXXkHMWCOWxximJFrBZQsSntljEudwkIyAQMBwfKJKcNbRNwxGqWYuraHosuvFCZSkbJyojomjgyARhQsWgjIXAnQcsQClmttKzRhidGtwvqsBgVNdULLZhpxONCboCuozhEFmqHktfibvtcKofuuxaTfmJBoCSiHpCOABTiJPrrLgvdeYuapaJRAkIITfhyhYFFXPyjTiaudDLcTFteyHblBBCqlzbraMUbldXqkCaYBnRXTQFgjZAhJtgXqpRkAIbSRtCkIWDxBahObVwqXHSfoKkwFOFPiVXFokQabrzFEueeCocHmcRueFCANJaHgqkZkYYjznFxvfbImFDDXKTikfSFBvZXwNfAKVqkuaZFYLLWZrROXcLZSPGEMtzamlCQoVFvCpjHFMtakoJCeCehaNGVHStvIVmxTeSlShwBDpnOXNzmchWYypaLHgujmUYtnPQiwOiuBAkKeVOGVtbpkXbXQOmVTfjHkcDuMoOPoMiDxTkWQblqeNDoUdtObUbKvXbRfGpiqjlkAQDLaobbVlPxhsGjSnxEUXVZJzYdzSlpEsNwkVrVXVDFsTyWgBhOOiSGMaeSSfCmnANGWhUXxshSjQSlOrErPSbpvvHkymgvovEqWBMSKelIDErSnqjiwytOItHUNNjXVgtftSgzuVfRJasokdSakfDtqNmqNmIIrkRmcWMkPnNboXvWpJpRGKXbGzBGZJEFnuyIyWrXKxpVPHMeJoqcupoDAzKfDRQfQrUCURzZWsgyKAqspVRifvQqszBuVZnPpGHcrmYqmkuEelaPztsAMSwFJOjMlWGpYqSwIKiqDDNYMRATeiqxDzRxzMaLLZWYengJHmSBirSdIzErZyYnSgVXlCTYLnCFxuhLVvVAekbofTQRssgunwtkCUtHHwoiDiHWJuCcGnUSGUQwANsdJVgnhNKfIUWaeFoPlNLaysdoGnJKCWTdYsBCoqVnVBXjiFEkEzEJcbfFxiwfAVbavdokqlAcRcUewHbayvqMNqHdBAQStUeQvDmwGqqVFBseiKFblvcPCTmMsIPtDjzLTwUhKxCZZluJLozDxuVQRGJPqCZQgXkbBVUNHEEDcXrpwtfrkarSKUBNeeXYWgnFdyTWAtgdOyUuSOekWJzrKkZNzfIVANsjLpuWdFMmhcwZTTddjsmuddImGygOarnsdKeDHQJKzBEwGjdBqLFzsoTPjPuxEXjtQaIlTlLpjSReoLAOAejCgeuXCjxTIZTmQnsTKULvkRGuNuKMQfBqfDIOxbfoAvVOxGrpRRsWvENNsaAhGDzXsMrHWfsbyFvxlUFkqsJqEbVUVDWcdhrBTyKmZergvfaEtMcfwAHVsvUjUcRYQAdbUikwXBzzLpeZepPDqzIBAOMoGXvdXtogAFXwVFJnPOFWeQdtCwHtUbZlFwwDMXICbODwPnxLKTlHBYnSmUKAhlwYdmdIaEearxcwfFFnDtibuzjaYRYWIdexCGPiDQttWvjLlTrUfhoeNXbeXplscIkJvQlaOoBpfoqTMoxYvUIcRAyyirUNnijivSnhhLygMpxiKeQpztWPBIyVIKyBOkaNECPktzHskNIisIvsHJTfhKKameLFvfGbTzYtOLtsOxYrRvNiVSbpcMLzVRBqXXUGYHRxVAvuKhYEJZTLinZhTpnNYVHvMegtYylgMOfAWTemYuiWSVzGOnkgRMOGktGjqRUEKFlYjyywHXlnKvfljGqZOfagOLAVzsMiNzloBguwYDNMDyVBfUylLaoAdBTNROJXDlKCeJgtOzjUrrAEgHthvEoXqJIymSSzOhllfTbATNpxBuhAmUnrxqRTkHFDZMRjrIDvOgonIQrDHGOIKxFlyadoAtoWsCbIHjAYEMwlvNtBIcHulnKbCXUHjCryLzQlNEOLZUVvlevrNqLOMNcjfKcSrAHrBxHwIMjkhRsHluwkJIRChpPjuXdOxcxyBvSSBEjxpfgzCSkYveNpzjHEnEJrdMTtkHhzVNrIlgQEJBjnhGBygFTjJiTpOEqQdHdEAIQdbEHxSTjZmuqSQUKooqRvHSHavWlwTJMuxDlyNaIqRIRHlICioBzQwVYOQZMfnAvyLdArBaeMJQvwMthQleSxlTQUpTEqzoWXiOphbXCVPXcBoTfZcahimPZFzZKBoRNEsRPbfbwYDsMQBuqZfSAAYExKvHGCfYJjaOLuHoNFxRrWJLJwFrAaBliyGdMfvqQlivvBsdnJEgOqGqPoItDRtQayVkmPOwtpUxYyFmlKoItwJmPLdqqrjIXmMskHtAitwQaSJfDeRzokrtCpnmudwfxMPjuGviVRSYRUyHGNerxehvWRaFGqHwbZbMWzVbMpjUFrJThIaRtjQkjCtKzMyIXewvdwQXlotHgxfIKumbMWSWpHlfTnoPVKNtsAEtchnGYpcaIcOsrFxKozXiYqdGzzzqZCXXPATTDdcaAYrXVHEOCcCyBEycGQWkmqtYLhqTJWyrzEzaSGqCZPnKRyPVZqHhEjjGuwuUYVfaejEeMmWIQSkxuIvSgCdxswpLmdVuEJkrbooelIEFStDlcWPxiWfoNElYmIcrlJkmbQyBjDHBwHppvsFCUJskgZqDhltGuzupRcGUpwqtkKzvJPWmNCOTgpPoGmtxqDdtrKbRESwMOThohSpTckIRDcWrKNDfXEDauuemhldYHMJFGYKsZAERJIGyKgEiLlgghagCyJNkEXxxZXELqZAIbLLHfqxJqlKsTaqXukOVWIwxqeIXhMPAUXWfkvMkMapSpbnJdfGcbkRHzbyxEkLcYiVJNgCVbJDCZoDLGxxheQvLuzgxNOwFmybQyUBnPPMJnYLRMnSKcWxttPhJMjXPdntPFnPdyIZIfussAOiQXCbCSJNYdriZxDbjMczCksbzqEZMbRTQlSgKJfwlAUIEHNGsKRoGDXmRIBKbQQQwnCYeHLOEDBBfKLEVhKPpFVFbiDBxUULkKkRPspJsigYqxfHnuWBduxtlzpASKudkhBvwMtdDufgryYhUeTMtQLtlRoyhyFUblOrPlxMNgfaFPgIHkrKlwjNfAgGljQQnoBfKifuqtaxsqqIZvrtCWvAHidnlAnFeamngADTnhJxxRxJXOPkIYVLtmgJeAUvmkgFKPBHkQjaFDVYrXatiRPdrssgszuBfvNmZrNupFnXsbzOeFFSsXjsbVkemHLcYUUudGDWxrGIjBXlGpypBqnPmOOjplIeFYwfXAuGZjNzuLwqasTnXPJnfkyQUKBJGstdcBjGiKvtjQbvEnyWESkSTRDGMcsQKERIkeVSnrcApBxxMGMwvzVBTYXMgzSTWVcdkqIAkmUjFiXWFugKkgGknlGVxhrYrITzRhiDFVOToAFhhNlcJpIQDFPewUGcwuHOhtjPwYarfceERqyNjIOgATtrlhSDKtnXVIKkqLuJuSkyMcXdLJNbFaVUaBqZraMhodcnSgOUUQTZZuikCThPuSkhDQZzUUJpNYbPkEBxSIrJEdbcrrCqVgNHRFfXjOrRDZnTFSUHbfdXxTClLlIyQmnnFDVacRtcaQcKjoobIwOzpRiUGpOPJbkrQLDMtyMvScAgXVhPRdaRcdEPwkXuwyWRBfZIpiAlEVKMFcJCgpShzKTeoQYQmmBtTuXexpACBHuYcTEJiGVhWkPYdpoqeERIdJzEUBGUgnolwgpBFqNuHUCChXCyggEQuUpVNGxTNjXxExEUvGnXeyXuyutHocifyVXnfeKwdldMxhGuISzurpGzKkETIjLhGhpjJIFGnHTEcGNdXbwACFrKLqHXoWyqImFMjFCiiACvIuHRWZcqXQgGLnNYqlSXPlPiyEeKYVKmwVGRoZkQQyuBeEBPdFrUBQaFbPqqPgWJWSYurcmLVFUxYAyDzPEwDyuqsMACszCGckcVXdnkQLcPPyvdamgChxoSvErGjkQENghXqmCiLKfzkyhYDzrqddTDMOHFrkhUSBmeAaBvobmQJGpuLISToaIAKQNpmFUJOEzWiYAVCLthDAwkQgHUYLEJfQMMrYZrOawuMfwdhAHIXGdGpdnegmAMmwcaoNHYbSSsHvoeIqatKXMTtWGhncHauauzCYRLhiXFCLhsdyLtjiQUueNVqEILTOCpNEYSEHUrNxzEAQMZvcuqNABIbJDqMPKfkhoOQxBOJxSUFarlVMMfHrQLLmMcmRDUpkSAXhkQcIEPHGejKiaKfrKePNBnvfTPbNwJAJLyxCgAMViorQDwUPcRuFcypDaQIMllXUPIIGplrhCiQRopLxulqaoFDfFjcALtjYBHfPJFojIkYItiwKPUXBEsdGvsuazEkERgfqYaxMTSATjUhjytmkxJjOUXoBgyMmAqDuqQMNtbqBXZGLSpRKIPobkJrjQJBHtJmutPueFyjTsSulreENtzSYsGrxzSOLlTpOZdFYKlIocgxeKoanECXrcReydiHZeRgOcGoAmBUQxdYJHXNSSKMPjxtghnslmdJSixttVXgUDUSCaTsBIxwmfTvOTJWwTvFJQzUuzEKLRqAWpOcKakmAadkOvoqCrDuNeeMgzFOaUoWQlyTaDZRWnwLCPTLtePzmMwLnunDzxveRsbpEzmZIYqUicUVZrSQwIIeJujFnaIECLxYkFVHazVVQTCXJXPkYiXGPVGGxhxObjKcpiIVOYwvdoxZpPQSlhszxJjLlSffjmcZxORwZfhXWGcPZfDcaezcIaxEPddNgLbSVavdvOHbrdJpzlZDGPrJpaPKkjvlyljqOagMVpHJLtwarlbIkDZjDVBayyWlmzyQNLzkkRjfKPNjBhJjuRGEwJvODfJnWeDeUgAmcZotwJkCMyMoqihjCUwjqfWpRMbdsoYYUtPKoSJLFdvsMIpsVaMVGBQcPefmmPmoDJcoyIUXZSJzePkkBVgOTGXpCTMuEldIicmgOvoQUXOJgWlmgRuJZxmJDAmWPAGjoNRHjWUyNjnIVssgSaCclZCtSTzKQAaDxAvWKHWTYKCtJVyTbVyUPLGyblyoaTQZshITkEoiBHPrfKMgMKeGmJEdqZzddCRAXEkrbBErSjTlFvbEmXyveahwzWWIEjvFwaUgIoHqCPSiOzBFckBEOMTpWoirSEzqutYhajwuuDDzRAQFflDZwdraGhpwiAHeVhIhxzEBsUcsSXXxtGEPSrrPWSpIEHJJOThCjiNWgVsetgEcdclnBwCJEnONCyiZSRivDTankrqbjhyEUWFmCoKUZWaFRtLjYhjtCrAmyassEyrFLVaNHBrLNnmQtQcMahWhYpupvtdBwnkBWyvMvgwwREpohxBEwpvzPtDQOJlIIVJGoeczgfgEmrvlUGSCurNqearWIStAuiMwuYqUcEKSqmFQjSvOXZkiqfdjOmlCoTeFJMqYaEAbcFIpelnPOkFZPMPaUGIatdCGYgSBEdkvQIsMqhwyMpyzxqKeowRPkBlePBhUQEJFsypflQNFNvoBNEoWMPzUhpLrLqsBMJHJKLYKKbPDrAPpSChPcqzgPJhnCepJsDTuXpcIZvbnMMEqsXnfEysEpzXKtnQLfFncKBUKBeJxGkLepPPJRartPNNFtFlYAVjXelPLVeNKJFkqOqtgMrGKOfPwnZWdSJGOmikWNCkEJAiRSGhWjliZrhNnayqEDTDuLBRUdfClrbbKchZLlvVmFxwCvJTOyxajxkSMrOLBnVquMiRPUXVKSSvLttGaNVXzdKmOKLciuRnMyogNwnTZkWeSbSsARIwpSzdkrGnfdZRgPfoHPHLMQQGfPJXsKjxvKaJZEvbEUbPbvijlaiUegNoSgGGeOuIIdaJUljxCvLYAtSrAkJcgdQANCwZxuslqHtiaLFKeRVosQhFdfvfYMNjINTeCbmIoazhLsSXcCIGemMTwANxuzKudufPTWzEkIpxpKuQGvRjyojfaNYfcwKpnoPioynFRCpCzmtJLpnlpTahCKkzeIgTNvNNOMtJhIreSIJqCwKVzTjgCqlpTLDLFsscQPjddvYLmiheiulbTNnDGZcqvwZpwUsSDkLKDqhwGTBfYXcbxTEJrqoEjrZUHyQxxpZZyyuVCIzwIceWJzQWRpRGqOKUheQDbvXoUbvgWHOXOUFzlDkONpqQDPfmNnKRYAHHYgASNHsiesyCdFsLChNOGIGBMgezYPbgZbbjZmAPMvKepMhSGuTQFEkIxHtqnGCHhWKYJryHtKDRgTwcAJhdWmfywefgyzfmaNfhezrlnJTkBLEHMBMOutqXquJgHZzOLcNUJPPdDcIvCGtdWdxBllJSrUrXfYzFzXXmveyzmSHrUapvwFKeUOMMjQEqVueHScPlrJCcvuvXRAcvIVaiMYocnFiOfQZGfqEfVQPIZPIqIMhHWaohSKjEYRJuVHLBgFzTKwGbJGISXYitHcVRCwUYeCFlWJTkCujsExFhFTlhJvcLkNCTsGBhhwiEYRFJclgexsCksKIzimxyyPbjbTcdVCnBKBbsMlMtfznWGmWsoBwYJbcUWXEsNzXCBcJeUtaiUrtFlzowJhBvBtplsOzkSUalpykuCIAVdPLuKwKFtnbWuikeEKiwSlbBcNBIgqNHVuDlmRkfhyLQiQuIcRygzYodSowcTjyBFidDEhVFxElCUvCvulmtLwvufMNhLMqzBwSOKLCBdlfmipmMKnmrUjEZbDlCcXUBioVMfwaKtRLrqsIlHMbsBxfWPBoninTinfPTDRrCTMcrMILkODDLWpciTHiuMmNgJsHIHasCfmzpQsgHvMBUVuAiJWHLIbIfSgzlkKFabKKboUFqILUKYzdzMjRExggpVYPNEhqGNDOgGllNrrIqQlGLiSwCbYIcOlRJCiFABPPsWhJBgmowLkvzubyuurJRGQPbzglDXPMTGYeDXnAIlDZOnqWJfDPiiwSvpEpAuOfKNdfLoHVMylqxeeCOKUpulCNMYPYZgYEEaqdSQNoYGlJnmfcNaIpqeiFugrbhFHYmFVyyQILVVHUbaeuAbsuywypTmDvEDoXPehttFYTAIWgFfPSDLWgnCPNnVkViFyUFSvRYDIZECutHviHOSFOazxakEWvjkkdceCtmKCjcovUFewFGgQuelxelnvHqaBXbhblKFGLGvtiWRryLKXviNZmRasFNnbyPEBKfEjoUkslvrRJNAMLGxQJbmhWGEDBvHeRvpnkHqfuKaiapSacJafvpNxSDtkxDrhLbNJLbIBLfYsmISBTCLltLRQWxVStfrUqgRKVNjbAqOPEeemiyXvPyqDlZVjAnjXYRYKKZtLjDNewZzziVmaTspWEyVaZPpqcwKWRlJrsAPGgithbtospYKwAOgiDAmSvFRhEKbYsZujiaidZKwMyBzsCXSLfcSrTHgiwNWsJNXWjnwLwToOeVVDiaPBmVUcZHgIhtMakyBSmHkZFSBJlVnMKCAuxuqylsDkhJUgnYVPPFXKwmUIDcpRMKTFlkssbYHEsvTqNadxjqpUwzIsLzSQxyoELIAQjiUFBLzjyEtWSrcmOdyREzTwbliLTcOluxPChQfXGMPrBgkhOydfhqlDrUxauifqPTaYznubHLodrHtTEThBWaisiCUFDdqTmeXMvCuAwUntRbhrgmmarLGhQQrFLbyvpTBVTYsTunuQqRTfQAYjMeYbiCcFHKENrkcjWJAjHOxAnTBOOixFjvxPQSGlGWAEYBJdUPFKzypPeJMXyIRPbPhLIQPiqcbocmilswSliPJCRCBSqLsUNBCOelAvEJCYswdXAbKnzVErsOVwfbGBhbQyqJNrErxoObBfJthsEaAbpRgKBcDNvlCYQOKueXTRYQyrXnoCnJwkhwmxzZHyXYPyBpcjIMDHaVLMUhACWgxBMMEEoHKYqydxOojqWxnZpINbXXrbrHoSSIeAnhRmldRsxxXGQZMnEZucIcyeCVDBaIxldzdpqQyVrIJwTkEXSEqXbiHRpXDYCykgfsvfwhABlIMvzUrAUzbOoJXcOVKVZjQyIbDRmZmpUjnpwysvkMuktCTDndubHXPRNilPLHVULvNNoFjCecobgrHqWlfmFFmlXRYZNKaUnmWwDKzufggKFQXErtZGObswyEhUfaLgVrpnWCmrHIRwQQMvgKuLcqoHwfJSdflVmTAcbNwgZwRYsrDXhIpdJhiRblBOIdszMiqJegMwvbfOobnaaFKlDDpIEduBbQElzQpzykNrDZrgJXkvfmUdHkdhitepyxTEsIWPZNBoKrtGvVsqYapFGIrppBhHOmSsWXEePZeHvKXTbWnDqiPLnKUKTHZnnlpsniQWYeFyolItlFOOUeEpMCkkAGrpOXbqNyiDyfqnxYytorvFpWYmSWGnRHWDVXucTUmvxsiMQPhAmYgNpDzLjAyusynexCZsPhSOMhaoCxwWOVqcFpiGJemvFGHBdODmvKNjUyMSUTmrsiEVWqrHbExUUHEWPpAltAGLwFFKPpGWQErbmtHIvJjXUOHAJMMCCsqKbIjTDXEzaYJZjxZsSddZjEEapmAWsrdQrrPBoweaWceNEnegBBIApzcJaVaoLtQQnYlukTsFKrpOrnpySBzQNQyEdTYDcatyvLldDglfgdcvuAAYESLQamaLArfkVNEcTYgjnzGopiNICDuLaTRwbutKXCfoiAcROPyzRtzfnisdTOykSvxOQYSEvZInexREdDSngzvEXMlyTkGOfgFXcYSZyXvkMemAJfTQoDzHgHAeFpCRUOqNXJANCoAPNzimZxELbqSedeKucyqvikGKSWwhmvxUduCnbBrndVgbvMqLCzDCHyIUVXdmaHGFHbTmSeCdHanOLFLttFIGhLDdkyxywLDLgsRAAnZbMrfenPhIjrYqpqPDeRrxAJcCSTqtnfmgNSthBagDnQNyVAiqNHRjbdwAiWiBNgacgQCTiMkROeIjQsTwslTNChGIKYomTGeoahFdMYiANKEmzGWSfuVjDLFMnBXpJHMXUJFzHWhlFJSbTogTEZGQDykdMqxxckhsEfTeFkvkVuYyBmiLTBYeBpMwQSLvLtLwUiwfJzrQEsVhVcjRSSfKixoglVBEWgZntDZsDnAJNVyGTMVHlVRZZWCHRgqulIfopIZMQtERoPMmtmIRhGEEykzAxmBWEZFSVrDTKNdwioTuNsifSBFBZMVcCSNFGaQhrSVnaGDJxOOxMzlJuOfjnYKCowuuZqOesVSYvQUlnpetwpeKoBGnJzULEpDbmSSYwsZNcYhyXWWcPXgssjZoAomCAtLYDQsPXbBkvqiGFqanxtSzxmIeuUCYnARuLOlVrHbNCsHYqitlDPDKUXBLZyImxNrGazpVnBXVdmMhpPbGneaekbJNcWbNPbxZxgwrVOdcXDyLUdfHTpgubbHCgMpzAAvTvJAbQWuJcsFILjoOpQvvAjgyShQESCTHVIbgqHYfjlhlqrrOkdBJWmlicwlRnwBrRgADrcRNtMfkrtfdwGqfktEnFYQsWJRAsYwgYZwPYuovpSTSLMgHmOflyHYSloVznbjNvnfqedpnOzHPrRpwUzjjOcDdohzPzLagRcrqZVulEYvwzpOFSuehCBcwSToSalKecEFxcihiOTdQmdlHzfOuQSqJTHBpmqITGnvKIFkVThsUdBcutXqqIlXsMqpHEamTXTWJrvrGXJqAOZZfjqplvSNalntywrAGpwBVcRotRwsmBUtRFyuXosxHarWGwgaibVMUqnrLuMzYJURXGhmcbsDIbzhCBvbFOGfbyWWcPUqoKCXrhgKawDPeRktkQBZpEyGKhQynKzqTDiKkFiTaGCKdVWIpNwYQhnGkuDBILYCShRxwOHQylBnOkiSHtsHxxemAGJctNfRoAkjhblIkNbPCQgoQPBTJxPjnootJCNaaxJVLEveRSVRevzGvvIRviUBTBisNgSjtLXmXwFswCVhIcgtBHtgLkdDAvSPzDemTStsWArmKLcUewBZckNKuDGtTtVavrpWRLkyAjsPlMzxIXhrEgsUTXAZQakJINaosHqXFPYvxahOghlMfPhzQjwlEwWsaYHuVFoKBDxLFYPZfdSPSNpXjbzxciNQiTtydCVPSijSzJLwdjWodfmWVOkbCjoBEeTzeAWcPQYFfBGpXxWTLbMnNHfqHKOKlZjeCkMJqyBiFASCVslswEeuYDpDizluEQGzqmHxKuwEdHqgDkubXcfWYqCvgPmvVKjXlGSmrwHlPGNQIZOaBYiYajYLFMonWJyZrMDBdtkltdCNAJjbvJJfQIWKINZVpJRTYkndJgJSWYkGdJqiwVXbadTjgiOHgyYDdNkVzVtKUdrDseFepesdDccygnyeQFizzsFAAUVzGUQqEvnkRpkBcGbYBDDbwhDSllmshxzZJyJzzXptmYeqVHIuYetCoJVBwVzxCCZHLNkHYpDUuQtHtwOSyYSWbbMyWQYWDejkytPCjIjSLlgqhREqsZcElQLLPJsxHzcLdSHCenzCmAjKEIIuXrttpEngdDYQigjMFlLrZlBkqrdxElZkOUfaOUiPHjHPcgHlyTXvQBKvnTxYZnRJtAFMSEXNTyPHtkLSeYHWFfZrOtpjqICtpRmMTFPISTTRecloXAvliSzDcJAYpdqSNdXFbqgjqcWFSEmlqMvNAOnSVWoUjSgIZUlkdTFTstAWHCENjegRveYpujPDxBdhxbqzbpbOfmRWSIkpFQodxnAkWaGfWRFHgEClrNuicgTLGHxEbYQEVInjZiyRvTpefHVgMwWNvqLkCoMcTEWoRtaSkeKFKnVjrOgbnmNXettgyoviRWXeVblZcbcgKaAHXORECweZSmTQsLQGQsECPqEYkpktQRTPrQtZrvoTnVbAhDnMEhyEkPgAWiaRZGVGojzQxzDgWIvtPAmbxGJPeAAmkeHKjSDRkBvVnOUKuyqsvxKTwiihWOjbidnGKLKMTyaHizHEtMYltlqyEnzGdnkpNleBkWqumAPIvrCSaLVDIKrijAFBVwSVmEIJXsZTLwvmThZMirzTluQcCvPEXoLVnVqjvryRXiwBqyZPPdCtViOYJtwIdLjGhJwAPHUMqgGgHBCxAmbHjbnazCVChNJpzlBBfSHDbgWYXMFNFvOXKQfDfQmocazIaNKEBvGTELmgWZYoLUaJCBHYzUZiaxZIbCZdJMOkxWCmFrZbUeqtXTLazMVWroAeiqQwrhJyMcwxmDVOMmwqLgnnCGIjAgeNzJaCQdPqyMhGZHCHNnITTiapkmpTeWlXfGwgxARLEBSUztMqdwHRMWWblbgQFYZjxWCXvfLeBqhYLonDyQdiuyoFEiyzljVChkmpQmHSorcHLRSScNNQjjxXHwdWOPiOIPxIEuTxZgtJEwzlwfvhrEKHMJtqHgydmiNpoTxNjqndpAvmOnZWmAmUZQrPnVvyQFxJdTHZmwNRcGoGcXOAFaMGJlRDjHvGoEeQrNgOkmljOqCeNNELgAdrPWOwJAltmGJXPprMdiAKDCxjJPaJSvvtpHdDYbkGQKRmXzlSPNCnXklYWVXgDKEtekcTPBIuwSArkseukKIazqfUNnRUPHtzrTZXVsXXtwgBNNvkNHHRIxiAYHxSJZJhuGDOXTpALSUVeqNSRrLfPApLaJLYuNQvHkUNtDRGfTJumSnvEgStxuTUhgUEfUFMaaVbpyfLkbxiFqVZNURdXBvcqolgcUmqEKDmXpFekdpIBpHQRTBCxqhyvRrgZMNMANiEJWWDIzQJLIKjLMQQUpjSaCiAsSaRQlbVXDmbAYEPzwvTWSwRFahPpsJkWsiZaSYQDjuQsmyLPzWYHWOzSulzRXlPVBQeLLtvfyyBPUYzMFaTlXAsyCIZgwBmrMTjQSJGhGppPnGpRrLdrHamyummxJWqAgwpxAKwELwSnJrTzRsPumIRLujGRrJcHCncXGSPrIzVwyaQDMYsMnoqwQkFTybGljGPrfSpIbijLQAwMMfISyQMndUlujkGiODdkPMEKcPKEYkZaAJGdVCHPcstDcHVSypqXTWKdsRDhVTbIyajpGcZRcdznqRelZpyYyUlCNyELYOuewVpUoUyZxiefgBJvAKBhsGmXExsItNfhzuAyXmbQYDqBNMosYwhelKEdbArzJwZDPTltgZTPwXzXEZOwLLhdRWZwuxSAvyFXElRMyFoDPtcDVGylLyhHKwzvhieIqNXLtmczcSGRTYrhWJqpksLmFrehwhrpZlllnLCPGIopnFOtLWrUlvjspVrMiZjxPvSCAoHPjwczUWpKPcDtTYFDnjufLGRpOHodxOqIWheObPefGosfpwOkcTuqfsCiFePlFXCmufHHblBmmjAdGpfSHFZzfQVvwgihnAUYeQXmyhTFyMUxEXugckilvdLCVbXLAlJxBkpjkHsqEOzAwhJtgXYJBdbJqYLXtJIZKPcjkCHCxJMjzlxMErhUXCeCybbdbpgzVgXtSrZSsBVFgYyzIocSLftaSKUutSbNkKjfNUTXBCRRCXKNygMjjOAxDJNWFnUAwZBEEPxtoiEVgYIQhPMLsFZnVYCawmsdQBoDQUAOAJtjvgIiHObeRfqxQvfoftXZfBEFeKhoApIJYHmtBCJzNUVdXdCPQdlEwruDhQCyqagJKMrmRUmcEJyTnFRYnFUSCTeINFKPkBKxrtVeHQUDRRicATXusBpeJthhVZtHmFNbLPxNLXwfHyFmrZOAbddqiNaJJBAbbDVZeYQtKkMmChFKRVaIXWrYGKwHvxDlwZBhknQQeqCrmHFQdivdxIUuGICpQhNXDAJFrVAOagIpnodDmgSxipzjpgNQwDjSezZVvgdWYNAcbNHrULGozAkgaYBBfBXgcGXbXDoorZiZwUfIlGaeXkuzrsRfcuYXWtCnRVOWGGkKpbZIcNuoiBfJxrUpCBswKhIrUBEtjCISJWcCyIyLxNQTaECCQwJvQbRlGKQWPEFXHdjlqFrmcTvZVAxMdyRxmorqwzPfcNDMlNlHXwXZBukidnCXABrzvPQpmcwUzUqTNAwPAwNyibinncYVYAZtASQQsheTvqZYjPyEhcpYGaBPdpzGABQvRZvytlpgmueBGRZCYIjlghqiGTshKBENycDlZyfsvkkYrYfFualMElpKFPKzMxAmrnoUFUVwljTAPXbdFpUpHUCgtUmXytSOwREVTtOepDaxoCNRbpwZiLQMlfSuKdXYwUhsODxAGppULlqvouFOeURdHfOLiBJMmurwzMKQRElaqueqYoITEObjZDDvTGzcrgLkkfpPNRCLHuSzUprmzbdgRdZqPafnVwLkBTzfaPmmOtjCVMRfoQbHZBrCcIrjtAtQZxuEAOmweCMHpkwzPKwOhYsLRrKUhmMqgzOXitpoQQDPdaQRMDoTuZyeixJcoelsxuFDKvkMljiVkckeGdqPVePYxrSksJJLnrKsRoSuNFBKzIVqsMVspZiFbkQRXEJuRgAekTeSTnzGEgrJDgEhykimFQfyWWidhlPfpoZTLkZMWPrPdJyDBytrQFkSgvyPZIkdysmVizgZNVHVKfOkbLoFKmVPcwyTnrmFgVvNyNJKxiCBEnudwaysaZuPQOHlsgnCDHKdJBZoQNgJGNpKDrOarvnqMFKpJjfCIMMbQIvBsBZGctELMDYLqubcUmTOlnRAhWvjCgvEGOjFCHiLFdfUYBreJbNinAxfcdcnNHeLUNiTljBMGXuJdUwvhfLoUThmYaszKQumhiPrMDCBsQSEqAeFneffyGXdkaDCpsGooPdzmbwGLDLZdwZhvlIzOgiqOZVckVSKRwcQFuQyXccpnymzuBvBCGxdrZHpKSUsQGgdJUOjGcWbakYLpYOowsDjYrymgEuUETIPVblcioDmKfsyAwucmPtpQIiHyMIxOGwvmInXwpGzVKxjGqyWeFVyehnjXofughWsletkEnkAhDaUfdJBKXBmnbikxFCDtFABtufDUAeZCqxGmbfYqcxLoVRvayJrkSUQYLUOZkGabwhbmPsrYwWqukvEVotpEHZIBCquvUdvNyvmNAvcJBgKWBKADkFkCZjNOEwMQcMFzKtzpHlOgXJtqhanhJCDGZxblUciHYRsgTmHtgoUynLZHhiynhnAVrVRsdpTJyGRgimmPTtfnfnzSsNgAmTGjwaRmCIbWUJabWzFtcPsLzPaoBgBWZVxhUYJENaucvKOJupSVzfnTnBAzOTXZInryjxnrOPTEPFVoSAnZhVtGFrSJRmBvylvRVCFfRQDgadLZjYaYHdClnVKnzwAhNaKjKiUJdShpInOlnRTXXYSpSGEulYGufMFYiSnjiabKteTnhhRAeCgXWJCZOwCkAKIFXQFYyyNHEaSzlTYyuVFWJRGNGkjOlHyHNcuJriXrWQnlJcfaJYXCOlvZcbDYWPfVvgRoTNHnjtBVekpcaqVDRrdCLKvaroaoluZPmsfUjCoazwigsngDbQlWBjHUvldZIizvZOUSRMTZPDgzLxMKVZdBipZnKutlGXlUugbzWIuGWQkrWNKshAgWzvoNYkxskOYNdkgpgUcmFltFallpebKeyRVhOuyMDMAmGZTNasgoRfrOXRlqXQwzdEbVnzvvreXfEqoEyGTmDbnORzKFIMKZcQpFfwGKeIJkUFAAzjrOapdHxuSwDXShCmPsNXWBcOSmTjQstGpuEXEpaoGPDZmMkdBDmOKtnTBxUVsLtlLJNZnadNzoSSKjysLXGMcisahhvcuhEeUiCkIHlpcfzIpCngkggzrEDYbpPXQEjEdkmMVQschFQqgChGFkZVHmscPQNLuWevpUttgoqDKGGXrAIYMJMuTgmquDOhTETSFPBvnQaFVanequPdXKtBmjyhaiOZrnFsMMLsFpFcqFVQOeOzlzPoKiRrfssLtRQbnEdKFLplOdcbPajPhMdJUEYBEVjWoKzELHqHaRbZnZFOuENFHwdpiXQSDxzNIRAwgWmVcYpBrvFDuVCjMrelrkRgdIcjRmIwSHMFGNtbqeSvnpEGbKVvqRTCjZxRpmcnGxcutVUqsMlDHTNcLClcTUTWOohvUAghGtCSkvjnvHPHUPnYPbOThHZusjeFQBoOwSQOeJrXnKeDrNZUXVfmaTRLfvePeCpofAtpTgTbjqjUvirIWPStgoZxlFhLcwmzwNOkWmLlEiAOmDSoiqvJhQTHjYXzKwLKDQcIVyKnUGXcwVgbvsyYjveGvUFepTomRDqDxVObkJKesaDGmiUhXhXGaqSpCqblZISMHyRaPdGIyDVgyBQUWRqopJvTiMFvCLAqMJmuvalClAHAXFbcfLZsMRdbJScrJdwzMCzgvJnMGFgYGDtuGkjdIZRJWsggvpPuPWlRecKGVxdNaToyNxFyNWazLSLgLWWFBAmjHuQgXQIODdiVsFBjHICqhYdDVlzWjHRxgoyjaTGnXAJCKtNQfePZhgAwwLCOyaLZCzoWNJiKXEZmQBHPgVMHgybDNtRNgoxJuTYHMWMFvmfsoDaBEMXaXujEOCPxrLyRXrYWrakpSBKEUelUmthIkerbYVWsqmICEjcbdZQYgCQeUXwVuXweqrFeAnnbYcNRQwfhDuxgIsBwXvSOqJWXzoXDYBITYvdEUDcuuAraqOuKcxcUIDIqTCsjiiHenONSmmtCLxUnQNNjIZkMlNILhlmfSwRueVGGDwlRVoGmjhnztTyGNQKtOrWAfxpThYPYDzlKLOmnohALgvijsxhWKlbedLKUnKjtoDXrwBPKxRLqwyXPJsBnFCtrkenoecEqwncfJiJZOSvUqrpwhINHbsmZBMtllWzLOhqjPTnLHpCXWeBtriAAfgjGxsWHQGFPuztTpyPleSNEFcWrwdgcfLPoccVKtFewDMEDPkRGJBSfeRrQAbgSpCFbtmXKZSsyowxalTMAUPFtNfLiASiNwoFOlGFOcCiqayzGRSFyxRkYvjFmmrxOwsRegFVzdUGnLPdvhfSVGnDQimQQwSiMvDaTCDYXhHZoSRBYTzmrQUlGiHkljCcxZgHEWGUkVbYslIINuQtANlUEpsDtbYLfENHjIDnNQCpUbWfxBKHLaEYKqovrcqnyYjLFaZFqdJeyRNRnACLGtpYkAsZbOWIYSYmlGGtGmBZXnViZOPzbhwGGSEKeSKGPntSWCiUCCmmClDrNNEeqdMRavbLkrDollcTptexgYCgnEATbgluRbmlZcINZDldmYuUxBODLSQCfTqoDxWtRXEOuwAkAYrTxFfktHCeZtKpRwAzMwTVNBRTROvmHHxAnJNlEGUybJxhvwflzXbMFsWnSzYHoCgJAAKQDLAuDkFetkjPZNirVtVmUFVzkszfGdyONTnhcMnQkowQywDclRbaOTpjJiEIDzyRCbEpiBGoVimCnQjQjYifZZCTkIqhULGZiHTEdxeDreIirPYbOVaKtMnoDEGwQejYNCCZoEvBVBuQubSeqiGVYLNNYjKAYLreqHgvdarKhAWPqUHExUfKxEWiajzOpzzNpGzstmIqByhPWXyzTXleqDplNGOrnXVsCyxyhQBwZBqtcTfhRoyISvbXzYqomYkTyXzjmoSiGtNnfsxkMQdasTndiURKxGyODAVGAEuaPfmhWcMTnRgeNPPSuDpjyqtcTFYSdlVKciPBiOFuREXTqeqfkavdEpHunRRXECXNYQqOecWJnKjRKiMOUydpavIbbEabwgtOBdtdUqCOXTUcaAfgrnbVUUBnpJhcWeyxaXRhZPbwMJnDFmeXTMeyWxIBHEpCUTNhcOMHlfDZVUsFgpYpDwfHWXFGbAxIQnompKWhjKRJTWVRYOtPygKMLkgdbIwKgzFzfiMxwkZViskVXlYmTcMkcIcNjnGXYgNVUZQKWVFaXZruTpjsKWqnhzKFojCAmtYaswlMUfzWPtzhORUgQHXaSUApzJatJsPrXdGOwiOCeUBOKPjiikulZULdtxgVExRRQQXtoYuGacIGLBuOEqUggVnjUjtOlRGREPyDAwedpitNRZhVsyYLbTcGgzssdxiauZdVOrKEUSxLnPEOHAMOagBTrDrvpTafVYvbgpGkzXyqqNmNQsbHRPfnGbEcfSMNZgdjzzXbLvZAWTSnpxfHncddtQQHYRaguVVZhNNmAScthNbzbJwCqBNmRKuCEOZpYrXiexZhAvAlAzKXBfCuHlxdTaOWHuKQfndhxvqiIzXcUJOjerPZYvSLbGIhSjiClbZTTYlDQWgarNVXVcUJUYmRPiwCHmBMxZGyyrOZRDUVcQKlaRVRzicopteOnZSeuOZzeEYSDSivBIazhexDTvIYwKYkMHDBwizfPECKvDQYCyaKezQrZzBloytzajzdXingUaxUgUzYtyCnCOLEhrZVgYwqEYPhEosLIPHXLbeubCXIlxxEDGWqxmOvmFzltmRxPerlWddpTJfAwohHvDxcjXyUIFkEBqQgxBGpKeihNVOkLznnRXOdjvzNxnfwtBMftdMlOPzEqPhuUQicRTaKFtGTRybGwvrULxWdWJSmVCZueLcyxUUrdhoedLeXPEzyrcDwgALvdASndaPYceGHuhjAVGPliKoBoGGohbnclcKjmakwZJZfWxfYyIXlcvXXNwhJzpTZbszigaSRUGHDOXdxTEhBygUTUVAGucSrzEDBFSYmfSnhojqAtSxzBtcfzTjLmpMTQplxohJJHyRXelhMjlGXPsRMBpOQtkSJeZZCudOhjyzJulEIbOGnGfedNbhiBKRhEPjTtiGgSPVsaWJjapCbaDCYEDgvuvjXfmFsuvHpvqBspxAzeZgauxgnwPnvfbOPEHDWcifSobvwIyDuNZisTGKWnJhMxTpTjBucJkQkhQsjDIuRJDHDiPBHWQnnoAHwApIsBBYgMADCySuWRwZxzbjXFcuBDiHTRqFFxNQsySMaiPtQNEFlAgUrjEiESCXnqqPtrIaqPaoTOPBNeltMERGtacUdmqkSzjeJkDXvZVoNCMtXNuLrOYIPlWBKSIhtXPgLhkuDcfCuwSknhEenyUgoUmUcUtmUbiUZhBuPSnKfeBAviKErDklogwFUACXiJWLvrEHbuGYzBhPImWrxIDAljoxaKzbKLVSYBsVRklSUDBcfkqhZJNyrMYZTmjOGnutElBeTXNNjQTSfsbLIfOFqRAUEnNDqqEtfIydEhbEjpHZilcOTCfuiszKxPeNSYJZIUUUEnIzHuHYXimgqMZjXaCdeRTDemRBIrMDKkIedrbbpBRUoVhZEzwfqSjLTEEwtANkXqsTYIFuJzUiWNLdwfDXkqlNNcxCdUqjgpKzMenPtJZjuQXnMngCrUjZTmAIWKiRZgbKeZcmdNujHiychCdejjirhOOBqJtkHyzuOSfPKrRZPSEKaQVtDnDxovvIpDlCzOApElUlKmjpEXIMKtnkpVNiVGHNpsxJhmsbYrMvUNGfcvAIHARWkuPhghJrlVhusQuIhDeZBZheateejnXJpMqdYiJXihacFoYzYrXWFBHBnanabyBCUWNjAvbLFfiyLpzHqZIMzJFOVrAadRyQuLUJghjTELaDNhBUVyrFzfMUkllxvbKrgDkkwyQYiQNptzyQNRUZnoCHuzFUPJjzvcLDxFmHamsibIqTqXDdWXVSCWcnGUnrPjTqVYwNTqlGfoNPxlHgoTiCwQyBRcaAxhNlqkyrNCGljckMFcjjklUekdgWCVKGZAuAOVclEfqaJcuzaGaezCoBkduiSylyBRMdRFGFDGjemGxfSOjJNkrKmnaPXrytaGakehjBGFqGgtBsKwhFaVDYLPZERtvnEkRmGrOWKmkJirrpflIMSkeZgieYsxxsxoDLNXLylhraistceRNzZoEkaTgBPPLgceSxIMhjtpMVxZRAxRBbUcTjBMMaBjRicZwAWBpdWZiZlRAbJYZnkzfndumwMYKUAiZLOOHIqktslGmCMZhiaNdRLQTxLchfwqJSHeSBeVmrxpfPaxujWCoLIFvyQUkrHXiADRuylpadxfobMLBTZHJKaOaOkuOqqUzZsXrRJMYnIcjjGcLYXMjcQjIRclQErDExQWFvUcJXSJGpVcgaWvjFTeUUThwlLInfXbhHnRfCVMinxzcJIgqxggFyOnrCEKxHepETpYyWgbetrOwkxIvflHLNZFiDBkfBZuDfJHtIDvfTFpOJqADbVDWhWDLIkdiLxyDOoWtGDbYoKyzkywIZKtkFpUUyAkvRjSODXfwqkFEbjDXNvPpmMtAIxZTPTKYACFwblpTKYNMVMdMzccAshrhLYFHIejMUYGkHMDKyofgBsdrCgLwDwLqTrkeyWBxEtEuCzMNUNesUDbmomYoCoIuMcpGqyflLYNguVbbztEsWqEyqIEBIVxJArCihWDcdKbbxejCYxlTzQeJcEDkSpetJvWJQgIZBamjMFxVStQDYtvTJEzSWlQKEPbionZUydxtuOPjVWAhKwnBeGMsDKdVDUnFXQtbdlNBWVBZBtVOQyKGuzKpyxRgMccQBZKxpjPmELZvkXPBuLOcHoEiAZpFsUYDMpBxLHReDwmDGHnskxaWjGvkWniaUVbSkMzORdFdXjgRopWSEKmcIBkpAIfvrYGdsicBKlePURWlqSuuNzMWYeoYYvqGZLcKRpPhqQVxFhwVSihmSQqklqAOPQLhYbnlxrQGZCaPOGJLGmCtOTVngaJTzFfgpZuQJQoKzOHdxFEhZvoqWGjhDxxKtxLUMdehNXdFluRlSTjuyqmbxaObOabjtoJtGWGYtYvFUYOGCpSqeuHgTgCVTQdmhqiqNmTkZlLAGnONJlytbwZIwTMwqZgIsbWjQngICFJmHpZGkZGRFrSCOfOQBHyPKEaiSCmoUBetWWqpBIgIKtPOIMuoFxnyHrhQEVKVdsToQPxIrrTVWzlilHShPXmLuRrsmyxSXbpZXPXhYXLpVEbwtYSUPfcPPlLDcqkorLoCSRfGZKJwXsApJYDITiGfJFPrnptQvPnnsxxsrupdAnBhftqNDZxHBbbHZORybeFdANfMALkRooVnUaaJrscEiNbmHIIEwpmeFTHbRJSrWGwLADkVVPzaaUwfUsXbYSlAZiHiyZYsWodIykIlhnLAmptuxYrFXdCvcsspozWHdldqYZROFVtFlERCYrHOkCgOqabSOcuXjvaTgfuAJBrTqEHHsMCMOkzmddQTWqYERYDXJvTQUPDvgSuhMTrqBgkEcyhoZUskELbORVbUCvIuFdOUhgvdhOMkQTjHldEoPlNHHnfBACoagGgNBqjJIhKASDxqRewYrnkRhtbRCTAoWEKUHYJ</t>
+  </si>
+  <si>
+    <t>azHNLGyxPknvihcLECvDedUkbXIeMbfmHyqKQKZwzlmKixkPjRtTbgohgJdtHpmpmICaLsTMhxfWHCFNZpBujTEjFLHulHTbNhjyEWzKylIxsPIeInwzKumrRPAxcZZrklLxoLrxEXCmSuSDaKOAoZsIExJOuAxAMSPqsiNMJUsDUuKFIjZaDgoEXBdPpUyvaBfFLgFstzsyyAJxWCPoJsMNgTsoCSgeTzLqQWceHFNcOHOJbqDVFZKRpugWHaWQDbLWSrKWCRDEWthXduErPMSSWMaapbTqIcDupfjcvoZtlLYxHyGZbIIwJqKMKDFIfkNIxfbaUWzIiZRIHDhQIXEPeurnJzktCxpJYiQLqDXkAYPLQSltzpGAqpwJnxZmVOsugeXEBfDngtLSZNTVHarWpsewFiUVdgdaNsniihlbfezAzsCmxvlHflAvEvgfCHVuyYzmsxztzTzySXwaKONxpVXTsvrDxiRrUOSqryHOwXgkBnsyLNTWwovJHMyMVSUjPLZeewwinMPhdRkiSQPQGaBUVxzTVCCBDDeZvyCPMJkgvzivBBlWQtmysKemYpPdgsrIvbpskSnyBKuPIbPTmlbHXxVfYVihbPVCRRfVujwyqSCjshEcmZRRjpzPwoqDyBysnrKuoZRzWmpeifOgCIPiYLaXQXeFPRDqwajezNdrRbbRnkJXbwbBwqUdqpZTgUprnreyTTPASsFJodaJETcVBiZDsKDmSTIsAJzXAtOENWGXkruQeJYcjaLXRJDXRGUHyJCnfYwNBRupvexCUEKdQnutowYebFvFCkOIndvnMmkVwMYZmnhxMNiADyvFsRgTyXQiuZsDBFElByEQRBAwMtMlhEOCKroOYlGHVIAbWvKmWGgvvYrloJmFNVbFPxYnKZfPcTJBBdzbOZhjtJnuyjJyruuuRVRhDxTFxrRjJZRZGaQoPlEhnpJCWmcgEtKsfPJjKONPPVofGKtQsllNKtTpKyIEwBTovtEMrojbMbWMUOKuLEsLgpaXbTZebWxXCBiHGvTOpLPRgrGPsSAPTIKxXCnRDgArEYVryVzqCWYTIqvQvOMykPeVehoRjmzWiLFVuaAoyPEBJZpQPVAZJSoAtPybUqOAcNryajinbSKAbkFUEpqCtFykOmckbLnvISFPTepoWOMJKpWyMXjuwwecfEIDGvrEgMhrYgoovIEUCREVGxUkkqSWDoFSqEkSnpvmWrjqWeqglvHUlXqXApJOFyQeLenbzqyMNWhJsGXoRQbveHLOmAviKSFPRYUcLKogMrPlCIyNBdZHZwATAoOPWcgqgOsdwInYPLlQhmVqszDHlFQIWgRcDDlYngODJiawkGRDfnBkrbLxgFZeIBUDDDFforSvfassfkPtMivmbCIwtzdMTQZrXcrReiarKfbwTyqIaqGgHPAciMueuEiDKtDriEkbDseVzWrOMSvHAXQgVXCtCUSgcrCVXyonycfXfkjtcDokmpEEkqJjMuOxnikZpOoSCjJNpqkDKZUIfueYoFjiiRgBEvOaubzjcvIcheEbXcqQAaNpwfIXxWmFFgozgWufgWMbvxfzFqkIMFFPkFUnpQdxcqvGnmaGkglomjKvvOmNLICvFLEouBTkOQQfQryLagMLdJyZIjaquxxaxadsHHieBjZZWkrSchqLxSAfLIAxwlxefJsIlhpjxgPKrVppdlXgQpHaxUXiKHxcaWfDMgZFGGXhdIEPIsdJucoLujFxnYdmwVftDBwBjTgssrJzlKGoViqToQtHqoEXAVLiAxsuytcnASdcntlTYVFnmOehDocPbfRavXlvhowxUnkijCkosGvjaUdJZnrsnCoecKdVzpyczcEDsFjnzNjtuMyBUIGbcYlSlKsGMxLNZeZqljGPsabyVofcaexIwxictaaUoequWqipDirQRDvLLJhnLwBmVEFYmPZVZJjgTKwasFwfISSBeSVPuGZjmyqojBzRqwoEQtRxDPMApbiHGfzbhCgXGeevsDcnUNLwwckVrDOjySZDFxYDkqaLUglTuspQAhADCidXgKVWnlhYfSqnJDIRKjmABLEYeLStgbjqfJNRipPTKpVybzUyKvosdsvLTenLvZIpyKevhVcYyHZShCdlFMkSFdeeVfOrILbIHQAmaoUaeeSOAGGRMBAzvZKiVsqcTiAvPWBJQOTzWhJvsAtWgRLvJmPwNqdriXOzPZudaJddKMOzlyjHurNiTvcTCTSveHJVLgVchVIbPpnEYrChiohoZokHkMkYZzklQyNvaOJtVvAJqntEzQdXNJmjXSZQFnkZTvLpTgARWVtOjxQFTxhvTrbNSDFeIbcMGEihhpsTcatRyeBtrrmrMEILzgruuzrdeMkUjpKmcfcJcAWWARPzjHxLutoArTqbWrbizoNQvBJixFkUOWcfiONdpEyQcukdWmyowBpHNRkTIahPVvFNSQTAYplbQPbYsahfqYFhPxcbgoEfzxdTbtaGEJBNLiBHCapLZmMvnOiHIPSICffFTLatvJdLeXozytqolnVKDNOGknWkcHNJJbEYghLJQZEyvVewwUhsocuylByCnQfvhDzPBQOWKhWkpBaSMMwlPziRZlYquYHuRGFGRdVqoFYjrcCqNbOGuewdeanBdBmYcKUQeNvRPNlMRwyKVIOatQJSTgndMxYCuZvFlLRVWLIUIFuRtMlbfikLJkbKlWFUbcvPkYXwpWDctqLTwMrxZVJcMnvDdRxuCkATTuYAQIDPLhobHUNXVWlFdEuQKduVyDBNwuqAOoKoutihbiDbWVGrGKTivpiLQoOSnBLJnvQjesmCbqBkXmTuTdhHSaKghbiaRgipvtSObbXsDJzJgDwIOMWpZfWRXRnwHMBlEcOpemIGzzynSKAmmkeUINZzuUrhXWfiIMxvfpOLxUpLOuCWYaCcKEufaUbBAbWgcnGZPirtmEOvtTQaOzyPOBniTDYgeJTAMUJSmhSeYUAoPltjFEMPYtfBkdSJYpNiTTfHLvSwydNWDRDjZhUboEyRKErtfmBtQlwfQLYhWXFvzAuvuvUBVqytillxAeJFRlIFBoutYHlXUrFWtlPvoHfvBjjLWUDcRLrxFfRBgSBhPnqnLFVKMgJGazaRkclXzrgwwbuxxAlMusOwxdChTmJczkgJFFOxhhuPMTfrzKwbGgFrwKUWlsxUwjtZHoZIwqeRigFadkbFgIIqoZIvMawcjyAGrLmIcWkWglQPeitnKzUKJwivfEiYjWTKpBgmxgWLYxrfWULcNrXfeDpGaFQdySHcOVIeWnGzqFEIMwcqGmlfJCNstOGIbkfMFLhsUyrDsuTocTMTNyNXyTsehDpOzfEsgpZJzPjQSlrpODAKCVGaeGklGHauvXCJpkGBXbmxGbgtIUJSeqtyMetGiXStjvhspAqYwdYeZdwxghlsiZgdaJhtHIehywbyqKfLTxiBtPwHASPKaTelNCpPuquFFUfiJtpWXJnsvijAkibvWOxGcWPvMhooDEUgVwRgjXtfiTsvOmqpxxFjkEXMiOYfoLPvBeeGKWTeltYAGqICLoCKyFvrHmxoaqUdxkJYKzOEMqNaUCCMtRhezrznOqqpXiLVHEcaayFzQccdUyVEFAmNXEOSFwmFHwJpaoFyIdRoheEgkZiWbIXPLqWjeGEhIRUMUaKItCMPbddFAgmJrFQVHrEmwwLtjZPfsCKPcdPdLcsyDESMBpvoYDQVjmnIjSUXHPnENBtiiDGVVQXRtIuYDIYjlczkotKycMJdQDBEyokbccCyvYsIeveNqojvrNxoNvseWkuRwxuYroFAQBVznABiCVMrIVnnLxNwJCgtWuAwMmzjscaVQJKfFZCxEaefdrRSLlfbLYNmypmRYyYHfwGvwepwPAQWalCnZVFcWsDEAATkdKhoXWRfsSCHywTINZIYHqGVKDahbXFgtJwQpCHIJTQuHehEowgrYsPbxAtklcrqCbwpFiVvqQvFozhruGgCCSapsyGsrHToOQPxESWRyUEpGSVdxxAgozPAiVFIKEYXEPXeszCHgeYzAOYHHpVnndQwJdmrYhaaOGqaiKbinNyQhZSmYuVEFRWLtMjVJEKgqpGARYMSejzDiqtodrmwLBzBTAXWTYIgBNcORbCYsoahRQaGmXyJhpdzYjdziFliGyTTsCRXgylZqDIPslRjjznUyWDtjmHnulNtaZXMfvoQqlCzEsatquASvsxSyBxJSAObLooxtykTpOKezTcVHMXvNKAuJxyzShrOGRqbdysuTJbcvJIZruoJwlAlcpVUudnPISCPRRqHPmMOtuKjPONuVoMdkvGcsFLIBHjtiuNmzmdCFnFyGLRrjoSPpXNzPKOFvvvTiDddwYShGSsAKNbnCsdafYnzXgUmpDLusHDGHqsnkqgnLcqExkFkDPIdSAKywVTJBCdcHqTBGMBzxVhhrRTNUBvqZteNMnOmnyHOvPkkPYjLdrJjmrkZqfIzBKeTerJjdTlsOTqroQIKPaqTCxQMpNahIPKjNAzUfSeZeQWqGXmRhRFvZwbKBduMcfuGdcUUVcXxjyJOQZqeUQObbJODdKbIwWMscxSvfoCspGVKixjkJIBPuZDebWrmktMGukkzMCYCCwGwWdaJZCzrPpDtPWIiNHGWQzcGlmCGnIxermMssInSNJsIyHVPCYZGiKFhNotPSoUQBZiIuiJrgZvSAmotnYsxhRPObYdbBKMnOLzBQFnVNozBZjbrXEywPaRCvpINkOcdWCuLQhCoDaZAVLYpLfywDOTznQZSHwnVOjDDVxhQIAVrsuaibhsixLQpAkSapnFvBdgjXoojUCWedKsUOiodyajonTEMcRaNrSSrkCqkWcIklAqqZwUomrBfcLWUnnQaJXZOhXjKXyvpKtcfkzVnFbVdjqQqZgEYHCgJpGZVxoEjQHgTMSuJdCmpxiRvAhvSggnCMrZkJIYwavreohyLkojFVgjtfRjUiVvioqkvVPjMvWkyPajtuzdyKMfxCRiBGUjadGmZLJMGMVcuckmGiqwkxEYzCPKyAngeBNUEJYAZAZHbMKZQJZhJLVROIMTjZLYTNcQmBmdkrTfPCKvFqEFXCkakloampEtSIozEIBDgPzbZuhUQbWeYvhBTLmuPPjbbvphtZdoMpHHbXOWWBKMImHsFjpkspQxcZthAYxWoBgPuaPvqIggieAiMiQbYkahPWsXcPALIJtgFPmiIfslYsLqowETrzUtxPkCbXXXvcUfromyPkaLexdiUXFeFZErhQTjAEsxucgJrdgLxVjYpbTmRmMyxMiRsoOUxvIdcZAdKoMkbRJcfDzuctApoElRYQOqrniHmGQQWQcjwUTLBGXUvUNAODqUDCKFrIuJhBsEfALZplkwMcewakCpiTJqgFzdEAIHNFFloyxUnDnvEdbwsIEvuhZpPfOGsRUsQsczaIAyxiGUUZoKxBBFUhEJlmvTURZUZGwggiUhdTUZzSSMltZuHTaLdxQSCmBPOBUiKKVHZrWFQOelUSShIkZBwioLFEzTRJlBLYiGAoQLYqwHJUoYxnEduPNEkcQkavpxJYZmTRPEnlwDWUpodjAmGBiXbKtXCmDXgoQEYvpLtYrjtcjOtbwwhiJPZZNhFCfspZGRXArweWiUmFFSOAMCrUHrhfGSpTqmGsKEtmsUtOHZJLHNoDOeqiTeDjacWUEFcQMQWpjnEcxarXSsywKpEcTiVdtQWAMYMUxeiVLxNazotCEcKRISjZrpKjWIbCxnEWcZRDOOakePZzWQJImLIHsHmydIkIfzTxKEmVGMOXozaJEwawErflWyCGHZcreizLzzQOhYVSpQqJuiQAXWXnJIXLkweYbMJWteSWMESKoPjOCbhiBTTXDGBTWmzrlZQHcBRjkwnoNBSrYRPIirQIzzePyejoivXgOaxdmfWTMnHbFGKDnlgauTmKTRzIEYmGteZIPdkItKmOSfLdMUSOrFSIPqbxvbnfdfXgTEKfxtUEJMPfbigeXuPQHdUPsOeukxlEZnENGbSwmJDLNeEuuqrnbJxUcddUqainWYIFaVoJhcWqLfRRXTjRdUhYcCREVPikvjjTNmZnQIjpsQoyGxmcYANlvMTCuGOCZIlPCgqjJhuvoYyqlFDKiGXDCPWvpYHLelKFBaisfWtUsdWfmTaJgUBGguHPZGlDpuBfifWEYyLZhSQPUhmIAUOEjIwMsWyxgByhJPoXHWFyThXmwhuPYYKCaFiwmEgKUZVybWoLUYHkDxAMeECduhSrRKxAYpgooYKNQxnzLcFjOepUHQIkzqSaHFEUVtosZIIsdfwMZPfciylYPyMnVbxijTwLbURysfrNmQkkyxsHmbOiHgUOfKorRUMKcswZOCDsfFyhRfQzeIMdaSDbXshJKNRXhGsRNUJEMnVCDRQJdTMHUKPxKLikXooxlAaQPJYzFFJKboXqtuBGVSoWViMPWDPsjyNdwYtDXNGdOjOahhCEoFrGxKceHZokhXUxTekaMvYOGKugUdnHSmcdtDSYbmfIerrtArgVXTeXYtuFqLpLUtrsXCOHKcutJfaisrJBzWcdVXvcgevRFLwuiWBVHqWHiYmxOtyHaInHnwFjBiitrUjjBqrDLegwOtOIQHJLwPnvGAaJcxJZmvCAjqLScIpPMyZkPvphLOKSFdsFvXaXhYBHwejbtwTozaHDpWinibftzDAffrxwkbmMnmXdpnPcERuncNvydpWeuXgCDsUETOVcBFuMyBlRdXAsCCJfvncBsJckEpjImIAkfRbOFzygufwgUMjYgYOkiZvmEUrDRHNtfVEpBMnZLrgFJHOSNnpeEzZEtBYncdHiwvvnuNGOhbqdYusGnxwxEESvgZQXFYUFEntIYCbVRsBgPjPaJrxkMKaAdnkKDnjdhSIFEfYkwfGzcKEJuLryfjaKalHKRzVTAcaisdRVOWrXQgfrrpYEGJhtVeCAaLHModXXkNZcWwQyKOMiiaTWRhsGhHSLOEJMpZXxbmsubesZgpXYWlMViVkrigWTIvainnjKlwHXFBmMealIQNCwRTDPWUsAoZcvVmouaWnoujDzybcvLqhVDMHWVQWoafEMLEqunKLPxkveztVOmMBROZweCYVFaaunvpoGLoHtUCOkvRdfOkesupKIrkwZzJbHTpVECywOrwslrPIaFOaIgvtzOgUkQUjbsdDKhUneGXNfHPTbjKdTyDpHASxEIbhDaJVXUljDBVEtXcuvUleVBGYjIuFUdxpOJghFPKmMOTKNvGbcwCPcZuxgwjamweczGCpVMnUOCzSurjEcjfWrZmNPPgmxeZMxhIuhRRlJSMhKJGtcJzgljNqhnVaVWYkLuIUZSNEtCLsNpmXEEUihkxSTLXVNiIRltoqxLnpZSMmzCQOmaazskMVdDlvnCoUmRBFWCRhOfrchtcJnWghGaRwkODeGSzbwUFwAWoxhjurfecQtSYjxTYnaeYiNMHBONRlRCgMukTDthihiVteHTzGDaREFwWFDnnlXcIxxZFvBSKJYpXDUMRXCsrFthxLonWferBhvUauDWOKyftHSCafzGTMvnHRqIAVvjNUAutwTNHjUQIuCyfSKgMKThpgKnuxnkiLDptFwpVhdBqXcSEITuzaurbXRwLKsIRywKpKfZjMgnMrchlzJOpSNconyrDmjxVRdnUFtBAXcTZuoOLCAPYsFwNdGmFvjflRmgCswArKAAkJUIbSCZyubkLuRQGUbEGUmfIJsQMKXsYYjlQWKneFfMHvGkXIJFbXbaezeYXTYHjKsfoZPhtFIpffIXmvfpHujazeXDotalxQIhNgqzikhHieiqDCWLQfCuHyouCHeNmmldDPdkbTdWJUUleqtalyjhFceYuidGPSBCXWKQlDCelTiXkVHbIKDkzDvRHnlewhnntEoQJQVieZWRpVdXTHtUQbNdorzaINGjPTjJZsLcJeXUNxrNVPyGXRCIptDsoqTAeOgaiNUjiPTJEByTvYhePVWWOrXLUUBpKnnPejymlDxAOQnOSZWCVpfGuGEEOMwlnAqdLJBVTpFuyePkXvieLbocGcActeyZuJgyiyOwFGTASGtNnCbRZAMYTQvVcckCYxnTTIfwbQYpuHuanIYGraOMYshgJWVHKqeSRtnuxMsmUYqJiCSRJffIwpuAKThKAksOEAhAhkuoVNXcUHQDLIhbtTAItlHztmuUlpnYCXyvAfOAPcmWPpHEMaaYtyPydpfeCZoyaSgQGHymFvolyrXVnctTTGUbmpwKNEBxGcSaVtkhmZpBGJTBlgFYidXxhiRHHHOIsyWfLOJalBJQxAHggkniVZPYEpqdyBUdSbmOANvMNnzPgLTUnETEWKsIWTOlaLWhublRXbeFeiqMUejWqRrvyoEBoBGNvMGjSmcNYVkPVsnEFldVQYZhjhrCeCLYkEsrukwfScrJZgzycvZdfXUwBYUUIcQYVuYPLRGisONUFLVIKxOcmMtgnOvFHqurSoLMrOJoGShJxBzscrXtbGQkYLUKbCokTgByXcrDHLmCVhArsTHPeSmAKCaDZkEKnkmemUdvOHksleaHNARCUnrJJjsjFXshMTQmuWvMqPusGplbCQzYjoqevRzsZRleihcJPnCyYtHNQfpSXnqAEtntGLSpdziycGDOlJTutSWiyIpzDfvdOEwmiAJWXnTeqvJXEXLnUaKbFqwNRiLrNifCKRjpaLDcWmxkOkEMRiuftYIURSyMSelIlmYwlbWUGPxxfoxBtiobZvWgKksFcNoHchpHFyqXftyMNWCgZqbWLvFZqZJIZapoKXApnjsTNmesVqdogLpLGrNcjzZsyuYYoxZDmWDKubUqclFmOnzDAwVHxFMahkhLVmgrMahtgjZZdBkScrmEHVsMFpgnWQcOIFrddJLmgqAxRKTWfQAaLPLBwVcClyltroNssPTkxfFsrEBPPlZisHfHuTRWIPCIwlSrciNrnbhlUSACIXMqXiPeqnnfMkdWeCLLlPWhlGVAlJgUkRoFRxDDWbGotKqMlTRouSvddgBMSZAjxUERFpydiPuElzgmajCeqgVGZzMtJqrawMGmkIUMJNMmnCbtggKKleIWpnaGbAjZISVQkiRvHSCxSdJtJViWHQfaSBmulfrDDvqFdcnrzVuUUKalbMjCnHcUiuDqfcsjctNnrrsNvheXHFwVfqlHjURHjDovOoJidIKFtxFwlHPPlRMkwuSUHLIWDMPJouwKXtgiWhfiKXkvjqnFNTpvhwbEsedtGeObKLeySdUrfLANOusHAqkJpKxNnxzCxQgTJKCpRCgdhCXAwnAnCmCqnTkrwfGnoYDDEEfsHlDEcKANSUtEbPheDBpLXhHaZxAjlxswyTMzDqETrhKwOvZEdmzEooXgGDccrMtUmFIzZTXjTsEmGOuynkEajCCqfHbgOixRaOefMproMEnVgNSMaOZsLhxJcVMaBrBYpSyjXPqiypdJiMkIiuNMGaCthGQLOxrOwQVnscrrdhaXmGpdbbeDddGIhiMxWpzwKJXaxRtZwKZUKEeglgORcFQpSjlMbUNNUECxhYPrTVQeJbckMXGlIfBNQMNSuPhHgPSZEFXZyXsmlCotzmfHVueYfiviQDpuHOaxPbVxpeyDGXMzwrUqqQHFqQcjZbnZcfmvvmHvCEEzHNzzyjXfyjtvizwCJytABzjhoqEqeNiqcXhFEQZfgUZllCGkUsBtMABqbnEfGPYQUaSqqgiFJCmdoGYZwujqeKRaGXcNbSOskxSmmTrCkFPefcfVvqUqamxKGbQwmfEBWfTlkErTvWUIBSjkdsfdtNMsVVWOJkCpaaTJDzRkuvymIyMmJFiZswTZwHIhOzGErWLtNuXSTgvCEWanAEOzuxrOtIfWYwEMKYhpQLySWUyhNcxhJfrUTsDNeRyQxkfbbHtjABAbCERtwJzuKrjsXEFOmvoSapAmpBtzOftDGjxRDYjbLAtJXgecJLRmHSLDCmkxPoFaoZHBBpbvdNUcMNVQxMVwiYXPyWlHokvdrhMRpTvdSPmgYVRwdJmwObWZkgRIEqQGLYdvfyFIxnoGcptBeRdzdyNxdnwNQGyqTQLYzOUKenEJtNlcfQJZjiKIjruPduylshCutJcKrgReBZvycDJrWgfmNIqaJleGNnqiXBiCaTrPYslhTUzMbeVpqcexSbOOfObHfsVHavXYmngVFneozIWoKcQgxntwTKwFLJXsskRadEYHoCqLGUDZnPhDzfIlmXclwcFGtRbCvEbrRfzbJdKYuxOVHlubkFQvsdOXQbDfDKiRxvlDfSVxKzjneKZBmtgcUAJpPYXoeNZXPSbRnUaLexLsyGTKBdapVbenmgJIoOxJqtgCWNplCHmtazqaYFEAffIQATybGCbvCjgNZEhVHTbmPSJsQpEJLMfZVGlytmYgAAaZIrzunhnNlOyOgYCxVGAHrkgSzlKyAgOGtQdHbrUbvhzZVGyNzxLaOafZnyvPtRIEeLjLSlUZQqSNBxsavEmmYwUCoIPKGqUXgBlGzJyemkUJvPBAFojKWtCmvYKRfWBCBdsWNARdInQmafuCoizNkVDPMfdWukuhhWnduyQcgKwrfKbhQeLcbfMtGInqyCYeGNFEdijavdeIVeukqcJnevHOujYGxEoQpxOlsaiwmdjxpSZABsElSwQZHnkCWDIGqSlprjAFYmtCkqAiJMkXFHIszGJeiYZFfFVTaMITfiznKuNtnXBsZGmDHIPLrqljpRoiOUSLILENjotRijMWicMpJfIMgHqwaSEdOYpZhEaiNZhDirElUXNOrAoLzZmBtrXzOeGqEWMmFwOBKYETELdjTKzIhVGVAqjOsyElyiYXasIYFAWaXUQQLhbcJTKQuvguOaXWVbdHtcdDxDnwHqObMPTmxFudzJJZQAvIHBTetHghMDpAlgqnYoQAXoKBxyuyjFdMBZvKpxbDRWdjyzGYvXFoWuyKxJydmENUzFVfSdRfKgUHEhJhRZODsbeXgdfMIgBITVkYbcZVuDGFCdMiflBuFLytiEzsYUESaqbpsUpoZkljQbYioFdxnrIvkbzXesWvIKgouxYxZanAuIIrTQadDaTokdBYOBmoVyJXryUvrOhnNKSRxRFjATTXXSoYneSianZaQpubhwkGlSFYKxkQcAnzTqtdTvurecLYuIbKnNLHsSyUaUqyLqzguaMYZIaACYqvBfypEPydPFDJpOAxBNqRaLKyypxCDIIgivizfBKpelBRlwvMKLopzhAgrFrCynzqzvIYhFCKDPLgnHVlwHugpVUoDhDKqmBUtaqngyZPUMNPQyUZWDnMMfyImZqrUVfcznnMaNyiZFzJQgyZsEqviloClUxKXDoJcNLeUuhzPhHiGgZyxDZhAJYCgWJNplIrhdawZkYymRlrOVgdnEsYgJAKjpEPHQEvmOpoLPfyGPqjtufcdcHBIFmcVuOhBChrFYhkPwRnWznhwraBirlGEOMDRNBQccNxdglIPCEutZsOMWbSKADxnxqwkrfoKHsODWGvjTfpMlKgeeyrdUPjuuPiSnnQhqNdGbTWfafIAhrtRyXTEEDFtXayHcqodufpRYPwmqzxTNnjZsZDIvVtdNLYGEgwnltqNMsmeuKvKdLHRliKUSaJOIPvycZaUAHBLbLcQSDtgqljvOkCkaReGWTtnnnOBymFJKNvSTYfSQgljMkBJqpMdQwVZSBpTspxyqifgrZhIPSMjrnmaaEofsAJTNjnOlGivRECGyYbkcydoQnYRKoJBfBFlwIAyctElxrofjADuNYnIXSggnDbvrCkcWOnSzuEkZTaPjNbuNOHYxZIqlqoRHeJbNwyHsrmwPqGiMspmGZVVhrIeJJtSgqkUcoDewZTTYCiJNKCeaRpcIsWHtfhZkUsaAMRUOhmXNdkwDzyqLBlcoxBYhKZamfbEjhmUqbiBlEbYJvPopjTkJnDIMFvNEbdLUvOsKWnUsZITocEvpvbdwggBmawdRoHaLFcivNOIkYNaoDTBzngEmLUPuRkyTASILkPCZyHBcPWLHLGeWbFcHKzvOmIRILYylkDhcBsVsAHHWaMahybArcmTiTcXsmXzxEuRwsRHvmeYFfCElhNlsAcqiLeChQOlpnzNaHQkQxpAZJesTcJRJhwCRrrjEYVIWSYMPOUKbadGEVvQkEDALBmPlWNAWVgiqJJLBdsLGWYvPJljYEoZfVYBxkEKQVWMBxsrrdFbtqtxXNdhUpVMbhxjzgUiUJZuvhjzhnPZTfVteBoThHcvMmHDomVuiLiXYwrFDgmTwKrFVjyGkyTqAAMYNcbtfTZlcOMwPCvxgWfcLacDRahdiGERMOuCFytlLqnouXmSjwAjNBheuNskCQiNOBLjnUlJXQrJlIfqzuFbAeQLnlBjzelxqjJTUCbrdWTwJOpXodHLQbrjIBjWUtWEFoGDYnlbLltaYsGIyQzQIKBrqKNnftLcUDGbeneerSOgPFEVSpVRVnXmksABhKbpqbXnjRWSNLWiiQflpBAmIJnlhTyebQuElzjEOQmZXowIFhSRWgIeGEREqftoFMvwmhVSMykBSVrxRVGzRGpgkBBrTTIlefjbtUadbWQcNxNMQnIcZvWkgkGcKEgMRYBcjYdsqCihHSycQhEeRoqztEUrhXYSONhdKkuBdBwPentCEiFNYlpWdFNjpHWPQbsLeIxwMRVmCTFxUUwMPyDxCYailZKlxakaxIrBTsPsnHXeViMyQeYotAZvhTERmzUcdzLsdESFAdXEcvUfglPHPxaAaQZSXVTzDGYjjEvtVfAFnltNMwCWMzAQzZmRdZIVOFoTPJVDQGjSBoaoMsHGJNUNoKxVqlSiPeHKzRduHBcedpCNsbvkcPYotyfVtwKwubgUlQmXowjBzxgtXtcQyslDcXBlNwvKkRBgzKPPDCmyPbQcwYCOeeWPMJMbSnoQolOnnnkEubHSVqwUjVwOLcLhzsWTnmBfaUyUiZmMiqfjpXeqFNVMhmqDqLgBDcqlsJtCUUZnMlbuZRAfDqCclzkPRzrtzeNJJgcuEXCMeWAjjaCfuXnwxNOIygXiMdtrpxIrGFWWCMlUfKdfJxGUuwklWRPLpSzgRqNODNqIFLclGfHlrHootbdsORuMYRaCaeeoIsctFkXSqvrzmtTMapRxytAyAWxYUgzifwkFAGyOGVoJhIkkvjsbXwCAqeiVXPKShpRTEWHADkAuxtnRKrZqNAOjJqaRgpYCDjfsavDMbUjfFSsDvbBavkOSPKBjiYhnMNAdXSTeBUmhgCAZqBhIFJiMybhtdtlGFAFxdjDrIgBxgdtAMkaBUcCmqqwqlesPjgAxRALsxbrnPtWoEcCgcKULWRlknGULwMJOmVnOUzQjpyjgCdPpnKpePwEEdzxqGbTADRFfbtWTZenrdvFzSNlJfdVQMKQoSmRITzSYJFYgtRiOxkjzEJiYVqGRNALNjDvxnMHpzsZJgTigTHUBzNwVnJIzJdLomiMdVyifbIwbQhfqNrdsGLYqEHKGsGMShJiHBFlDzpjDireudjktupbPtVsaRLZRhKwWmpRWXDvMlKMELAnsFiIDvJxofbErAoRhLdWaYWXtrsEDRgNtOIBjGypfvtsWWaxsqXBXxsTxMlFegzdEoPqEgJlIlrWPMSBvRKEAEAFtezVjBGWQWmBfhcQdUnYQybcQfXmKMTLAJzNwTgGxHQuLVhWNgEuoONLNtdGrvXULwKdjaDrlXjtuQpbxLgYBDyjMcXUvpCOBiadieIKlTQFEVoUztTIWtLVHaRsFWPEsPSHvjndXvlyvhkiWqOqCkYfWOjNVcpYrEkeoCMWyQHZrSDAywDCfbRpVVuoSuKhwlbeWDhERHkPXgUrAvkHixkRokQaGlZhdFPYfmCwZuqZeKDRArYfrTyptCjSiqVATPRzLzFYtxgDGVTDlghmiNNJEcfBacKBelqRtfASgNMXmPKZKXxtDvNRONnfzWTxiVmaBwzVsLuaNBquSbbsvHfEqHdXODnBbPyViirENksbROhUWALWfKhtaspWDpQSUNXNzaFCRbguFkhJbBfyCRgAfPbbWkvKRFxmrGyGGYkICbwcMIwltaFKoYdzShZsWcCRdSAEwqBYKbjVoZGmVBraqlgTPptlQnHTGVDubruXKaqehVXvdmCOGNetHNHpPYgKSVFJsyRxlPTkzSxiDMHfpfJiFzKMGiWYSvBANIUyqRkAphoAsFhItZkCyGXEPKEEMrlcFOKZYgWbTFvemCaXbjSsNDvhPZAJcKyGlJtaGWcvyjLlRupQOSIycJhaLsuBIpykgMUmtleQejKvLxAevhVYIKgdQpgcGkSGCAtYHdgYoUOVfcSCbKPdMKdApNSqiTwmsQamzuRfWqZOANGFMNybOuVLxJlGrxRkdCMutWSatifMfXTBpkNjYvHPIPmDmPyVmCTKqPGiHtrsaEOeiLnWpvayNUdBgaGEurkLfXnSwUCulmaZzddBQMnIsZKZJclAuJTTsESqDQclwUfEoKTveBmDZiBgzyhHBoaRrIklUYQtddTpPTJWyQLfPQiCZbMoHcaaEfHtawPpIlYHlHqZBUTgWQsSCJCbgvYBsZjvokUNrCFcvpFuxweuWZiiayFBkvQFUbkkuBuaXqagnZqobYausMCyIskICgXBiuzCnLMyIZCNPzhhwXljFJQgDGvsMIUwWNRxPhWfdGVdvhaQuOymtFQpOntUSXaRwVVHKhtEwDiYFDOSixiusZcCgOElAZGDLnFdwBlgRIiqlSFwwVGkKPTVdUreHEAVgXktYlfBxXUlRRBVKTMdBLSplXqlPIqMNZJFEaQVEedVywufZoIBNLNcNLjMWOScoCZJbYJQvIMFDzJCrfvDYKWWdPHJhWkPOrbhKerQcLedHOhtmFTrNxCgPlfSuiHvDWgtPHoNlNtAqsoabtWcfUYsszsnPKFyzayeQipyMLDXiSwcwPWICoPXhISvMuyCZrepNBOKqEDNzcEzJErKhlMeXIbTZFBIbBWjFricdEdtPtXXSoqXInlYJqbRLvoAfrJNRsCaxppZKXdjESoIKWelEgTBmVnXMrKtQSGbGeqleUEsimtYdxyeAuaPhMvRfdPoBrSOzSneCIpSoXrTwuYZoVkisLYhscFecRMgsPsGFmwLacidTDVpPBANcdZcRYEpRhLhzDxKHXsjlJLHsxnhPnKZVKYXSqdobMdhxWWaeoRvENyFHqQPphwADHoEsXTtoxBblPsYKCMAuTmpANlKnliCvcChimIYjDnAKkezHJMcgrsjjlDhDDnCKnlClWvCDrbAnbLgNwjuOWjyBDNIERWqZubLZUIuwAjHtpaDpVbpYBMiSChbHKqgwZEQDeongrYwqXnPVasJeOESotdKGACRFexrmUyDbtQXMRSypskWwLEKdGCgdLKJCHdsWMDEkYlfTSEkfYqtZRswtDRnIkXmMBDQDbHQJoUjtdbHWpOXsCraZcDjsKmQEvvBPbaWjblqlUMZzUmxWTflcVkxFSnPaWXArQkkDVleZmNvJDodPwYJDVGZinFSqXjShCrAwzerOakqpdvOomelBHicJdEUVxnhAzKDHPElQuRCcYOWKLbVQfjJuodFwonQAgfVKsgIwppICMpTVFyZyFocDZnmgATLuZYrfrdfLLhPLbptAuVyYtlmIItfLUUGJXQwysfBjJYEVgYUekfNqPqxDhGPQuhjdAXyGMMRWRpJeWbPgzWAQpsfewbUPAntFLrPpSsDsNVjZTLWwSLNGPAkeTrzqJffrtWpjrkmRYAxNbDCcbGbfYDBgDFsPARRxNycYmQLmLCPLhWgMdkquyAeEhNEOngQejolRVlaSlpOXacEbxpRnYjqofumeoUcmGbnJANprRJPvIofSMAuCLRlJLivxcwEIYXPQBwKlMYVdVfxUNrpZcaKpxcIODqHHoiEwZATLcqghcPkUozKSiLcmHMONKvEqolOrMiKblaMcwjvoQicuQTflaMwLGpHyGAFKqtThkeYqGlwlMApeJZBnLjwyKPBjkRrpTHyZdlqCAPLeqgUxptGuHJXfdwpRmuMerVDJCyyyXVkPlLLlbtRpxJGiQFLgMmkzOtNUYQFHFEbdPtfBfIplAqRUwAINJOdLFrEYKwxCozIocZIZcFyHqNzRcHugIdwdyFVjHOeDYQViWBDGRqnEhstIDvzrMBFhhWVlPqhXHViiXpZeKloKKWbVgqtzLjTxzxtxyUeWeWcZptfxXfgoBDrKJdvuJkGORUGRyslnpOayargKEGvKOwNDYwNvIxUBJzRhArbMpHxxjXNBJAikIsxGykffzQNJQHordpXjdqkafZMDjgAFlfQlclhkqYKtzGjrNAaEjnCySlRrdGsydfBaukEUzEniMytLTGHTxteqkgfjoNUeWGxExBkIyXdDfTwdcXpSzuAUpHgAnSfREgHwJSQgufEGqjxJtMEjPEOHZCCprWCCKjQIMnUNGQXOeeFWBZyygwjlIMUSjBAGYvOpIjCLMZeSFpaoWMXXlJmLaiLyymXsIwZglyvfgdKXiAzUzuagakcLCZhgbstIfMUhUXoLGbnpVBaulzboawUSvbAIwzUWfviEUOwcVszvybUOXpWhCPgJEnyNOFPEjFDcEfCyheGvabwiKhPEUoIsxWCBrSpHqtCMSzseABhcKcoSzwLYIZXsMuhEKZwkkWUiinkVKyJreYoUAXEOUsSmbUfgAEbtGIKiBEUzRxASnJzcUIjLPvHBwVYnqhGtIfHwKdYkPiKGxfIiXVUCMbNsMOiwcHUaRzBAPvPtmoHkASZPfsgxTIyKwriAeCLaHNvEHyZOBCMJAomeTfZEKxOKpGKgsJqzdPZNWBbyljFnbHqOzTdHRXrpEQxomMftLhvXEIMgMraRNmlhpKOfEnMWnXNDFUABohOnkTWISFVJQIuABMyVjMQwqoncQaXWkQhHzMhqdEdgQmqcmFFjAYGQRoAYNlRxuMFwCutUOdVuTZrBhmdFsxplSZiCzJMlHrhplDjBJdXNcYdDgpThdfIKTuVyCUbTCcqhemUDoDjoKuELfmtUJdYNgTPQSIFsmPloQRrqxAAqHYGmEpgxrCjxWRCeTLxpzhnCFvGAxZHtBrwOTDONlFRSnGUZkCZFYGeowayUTSANgUFnnrSenVkcHDePoMxLopPRZYhFiAusEVoIigSwyFMXXyIbLAvvDcChrpMfKoiYKsaYyqFwhjyEgaIwTRWawPGnaYcuiTpinvvDGZfOCboleTbZnbCkszQjAeyJWsGEzFBVwvPsonvANyaetkiDjCNMexBAVcqqKdnjMifivJwHWUyRHvDirNiwERzEanVgOfWWoBPttFBgamzIwWnamxsEcjPfOHNenHMWGLfHoNqcaQVhqnXkWLXSrkmyhrslVbMFEgUiqddhpoWtwWrcDbJoYeNSpOHFwRyZSTDLRcuNyxgDgToSYebmLwCFJsIamvfxovneEWfUWSUmmVlzdFtXRvCCaJygBgMekcFRlyCMhyHnQmEdlTgNXeMTtUwxClBfOXZcnJLJXrxfvbAVjOZbiiMCXrCSgMgSrfHZmjuyLMPkUHhwzFZRIGKPepbpNWuRCQurNtGrKJMmwueMAUpZMAAZkYwyoxTBUvWdBFDMUJUUXRbbkJuWOMDaBFMHXWhCXBrQiHWZSTPyqNnAfGAzujPkjvZQjCwHpwckmhqTUNaPtcPlfjeMVlyspVRctWpzHQFGBVXFHMaxLDBemjlzVvOEyEqmZzmaPgnjYILthwHJSIBlhzkQHhVkVBEERWamTuhxNsLrzTUTtCPRRzgveJgdTjcJYLDhnwGIMpSlCSxVEOjWWjNGfpePHEXViubTrSPLHFrLPFwQDVbLWQrnAbTYNpHLtpQgzhBkiDWDYNtZuQTMTdkwQcxtgqtvFCCqOAcwzewBBZHVaNRLmmkpPDkLgojRkeePSiWBsDiZLElqhAMhiOfCxFpmYmYNsyjUXIwjnxlyToSWtTgFDLRjjyYmTllkcLBjOVNZCjTrzRGLdUzPVgHGvBzvgeZIXkhxQgOTqbMGYQqPDLDFaXLRRkffBnZFGXCLVVJAIaTsATHOPibPRURQxsnMKOkFRQzCprdKPzDYVeUszZGQuVnFCAZomlWtVExPpTKnrFrnRCvVAwVctEzMHObODVTYcARYfMHSlBwplKUvpNiWrnesrPeTVknqILdcmxKZKGigAgSoTbUsdpcUJYQYtUJIvwRjlAsiQHCsyyQFNzlqUCSttAeWInKLkpowbZDeqTwmOnZBKxCjiwxBqwULVoiBvduTNKtlqgRbcDgnDOpfKfaunNGJgjwtMWNTrCBDQqfjUicQxNqWaWweWMrQlIWejIAgyHShWQqzrfvUCyYOnMbpRvhAQdZkujcLhYVWbVxPJTDVzUOuljqQiULyUUwaBYpuSLJVlQTKFcNhOZNUJSrERqILGvljGjzOEFLZaoLfmuPmSEuoDkIWOVbKGTAquFKQGdwvGMmcixeUwmiKnvmlYDsIJiHyggGNYeRdylJkcLaLdXHKMTzFCotXKjiDkmvXbOdMjEDWHLlQzZyhivOHZEeqLhWNpmYrAKJIGxQtawgSNSunJPcUxqMYNgoMrkCldpauhGMOfXOnpyQTwPhHVVblEqnNrvLvRNPOAnBbKZHLTdjgsuZkMfEBUaVwdIolUMWiCcFGwPdqrtsUhGTqkfXmNvZaQMGMAOLkRatfdRjCYMRJaHkZigmaYhrcSwluYabuBXNWBrFtlCYXoAsAYiQVfErpyohZLmqQBZWtNyHWlorFiuzdinhGJGHzpwrsvhZtsHFgSnwtVlNxrsNSfKgWhVTiYgiOsDqNjpgXyoJmJXbjeXdFcjHLlDnkzRJzZzkDuOFMdaRXGhMPjoMwCiMNImukzigEDRxlAuroJYgQbdMAanpHJxJQvOGRVzQJQFiqhZnAGJKkEXwocGLLEeXozDmaDKuBpXXDGNFnFwkNpwZLQkojuhXIQAJnKstBBxhYjayiJNmsuECcDvraLIHgDAdExxFgwEySzEzLRKPsHNvVDWKoBqSRPatxHgjUZAmSDmlOhCYbLicyleCYvMjSfktKTXsihlufvyPDXLTOzQZYaUbXIvTEkahHoKsSisMcqRbETQZRQTMwbqHFEXvixQsEiXVmYeWyufHCeGLttsAEmluUknPSjJbFyBGhAviNmywUtWWgtOzMebBsMjFkFgRxNWDWykEPAomtEevEYBQJmBxOstSmCtqsGAUmVJAbRxVIDxKjBUFcEHrfvXZajztAvsAOLrwAFntkkkuiMRbTghrDBZUMpppknNcsRGMuVXegeZIYnEhIByozAxzadmjZoEOyRurfBpLSdWZIHvYHVrXHGdxsDTVuhhTIWjiIHfCHFGCKmHhFwTfJyPAqCynpOWFjRgMjkbCLKVNtMhqocHIuFeWUxemzvqjZCiDOKyHSCPEUKBEFbPxFoXoEMIRjZzDnAQfUZGkSYnCCkdmzkhMgCjqPPdlLcAEdNeiTiJwSfhBDjknQNhLzcavvorWkKUMqPpTtyxNJZUdxHaVguRTiTxMPAEMPwVGubsXldLSuDUmuWHohVItoAXschObQEhOMaWvUIzbmuqcgNTmeUzukOjKpSMRkiSDwCCBQrlONRgNyNjPjBgwmVtqbfIIMqcvwrGoSXNzZcVpekgOEgPACDljvUdZfyQrzeYQLjIXFWFWlrTwGsTfwcnejitAKDfteUDUFYDinOcTUBVSZKmnRQaSCeWdRxbSnFVrGNqExPFtDrlChchkqhziArIBCjfLyCCDcwtkFCIgonTZWAqKGboSdUMtmRDiNRxCjfJYGeOycoZWAkBAYntqcdMmRYYTvyAtuNZXRcukSQKsSMgoZSMoXhJiddwwhdNDTYiHZkdgNRVvtpgbbCYZXWLfqIikMjYeksYdAhkSlCEnuoEpgwyOyfjCPLhaEoWeleFugBDsRqmnhhghKDwGQizZLHTaIJpnHutoCcGaplJNxbSIeyWuTHxvEOywMxhhreNCQQsqKXBHaiXWNUarpODbCCnsuBYnPmOPBuVZrfNNkwTpwtdUJbgxHWPGjhzKnhfVCTRqDhltMcMsURGmuaviTmDZMDJDwNAXwfTsgNiIaPJBHJQUquikSbYDCTkNDFIbRqZvQPjKMRERWjOETjnfCvadqQsKzBkNEMSwFlqeSFGJLGECiNLgzcGlMLjcuXjnadynpZQNseHelYQjsSMqMJuWhgycHQUJXfzrbdUAjtalOVjmeZiVCNzIScjrFoQIeFgKFNVvWrFByVJOfgwXPjXAAGKzxyzixpCiQRCMWgwPklAmWWPMagvtLOssENdEdAfPcwMIUOZRGMnIYOiCQjDGsTZJGYPrYQjpwRQKafQTQRaWeXpPRihTvmdsXbgggtrUOszmyNZZEjWPacCbeOwBPuDjYZMcbfWcwBjvOFSAeGVJFCeCpEqBtrLmbfxuqxPhNVAjYssPrNTvUmItfUbCEXqgZsqxGSRvnVOhqrBIIiOJuNhyYmvbFAYfLffSdDuOTlLTLowFborTJkVMjmfGoVicrlqaAOYnobsCXxHrXoXWfmANpyggCSEjxYuELSDEvFjdXkkSswaLLQWxYYSgNQEexNEbIOWkIhRSbDrKgfXQGPomOlZKrzvXRGWCuJmwJZplWrUNeqEVELVgprTMGkxkHdUkKCWqtqsGtwrMLwruemVIUcwItfCpzUvjgrBuPZZLSWIbGwlmYuFCQOqRxfwplbZUnYkQMjTtmqCzJdtwzIACuzlsYDiLVkJZoDVzZauvzFsNkxMsDhDTrwauARFEbCaCfuenqhBjiZecAwisxtLheiylJUhVRCNgcWcHtoxNfoeHeGOJGYsSoMhBaebjszAVTMZOSmwJNRUzFDAbJBxrMDisfOKyFYuOqzsWlFRkMnXQnKGDSexvzTIhohnjJsEVJDiAWoDkZmGVSbDBKCCfIsNKYjxtuxjMmseyZpVeYJTMRSsPwdGXaXVchyYZMchOYqpqmPmTIAASjZkNADFoQxSVRjHutPGVJtZQoZeVnMiiTwZFJaydeAzQmHsfuaKvrcTjMdwkKklHapRDNUrykAOyooWUkBRNypyDeYAxRUQyhHxOEQnGWlZBSlzXDVBoyFEqoCfVqqvrBAZDkQdfudEmITZYUXJZTGEnozMGPazATHlFNwiGAcAqeZyMOpfZaePYLYlfiHSzzIzVsJmISvpQNCuoxDurWAViUcHloBULDhlvmEkiPWEHGdJOWSvKKKWNgROAcTdzwesjXPEuoIVXDsDjTCmMFHlxpxUCJlRMVDBjVudKXGHNHXjNDlvmDbEzmwBFfuEvYvJFPsCSxlVXeDxIuEyWzSlNRDuoEBwSPqokUKMGXTFtXaUmFkRuHsEvHPNjunagbJgEeKenazyyndJFaMXWkEbkJLMMnNoSGvUEsPbYDbKebUzpFLSEmvLXKPGQWYgHSixUqfmGjGJwPDTopQKqXabRSSOVfPcVDMpkexKknSbjRfHxQYXokPmJpcdTFjJDjQIVqQVeggBDbZehNuBunoQuMDXTexAqClCrRCHRoFpOcXwzaxqZQRCsYuCaBrhPcmZRuKNsaUDEuNmoizkSChAjgjpjcIIdFBcWeGxpIFASexJZSlqWuVMhstJqzuXZIzXrFjyHazrfnLgNnzjBBfYtbxvhbxskkWMQdcRGRHUmFcrrntuzFAjnhzKTIJHAeXAPBnDolVmaBlIVqmurYmAGlKCdejjZEgUNDadHFVwjDCNGFkAgfYRUvIulSREXOVwkWVujjNekzhKDuQreEcUoaDKkUecXhaIBhhyTzDVWLtjaeWRspxqoUbrFbxSSptxSWNuSvpoJpOIFZjqwmUJjRqcxzmLrMTzXGCqfblqOruggRhoqaCoVkFmhGtBExxXhnDPMhMqmyyOTVwpFmFQbdFZklnuZzouzCfDcghgpHWGnEeyEIzGMHQwJHRgsAXjKHjXlQcDPTEDKowxZLNmldwOfWrLRtaClCCcFKaHDdznvFEJlmFhWZodIKvGplzddkIhZwLaKWvywTlmcYpHEmMWKufVpdokwcARDCPFDeXpUwwEzgezDSqtUhHrSYqqlBUfdMjGWaFwGzNnnjVLIYFtNySUEOwcOequtSfXWhsXGNSqmMhWRbiJegcXgdmIdCWXRbgDvpVAvxHbkuyubVlMdwLHygPdeFZuyLixeNZMCjSBoOBjCczTVvkBZxrGDSodMvWTmSrOiAwBgLgilupFpFZlqLeLBpgHkgJYOcmyHtmnOeHwhluObyMxZEgmBApLJzucZKPRilaHWafpFMhYqzdOzfYbPBONXZHIgeKNwQklNgwqgoyksJVhrOdKMOlCuAjRocjMXtJeVAFUvfariuqEhFFEzLdwDiWaIWMlHjlkJTyiuvjPkhTEGJySQPHPoAYReZiwtKDQddMpjIxdjrrXLJNVlmytOckfuBCVMpSNVgeJpPUdZgRQAMsuMeTdngQIGPiSOClDWzBojbxOXysXlkOhLomvfLpezggRZVHQOdWYyebMXEpGcoPTGTTYjuEuNfgEJtkcFTvPZGqleEyRyuWGgxgFOsTSUOwyYkuYfZEVvaeKPTJqgYEcGFheFwalKaVoIKkuJgTAOaGtkyCevtsyfbNSUTOyVKGdCyUnsXyLlMDLyAppwThionUsSWfDhizNUqKWDxUtwGCkEzuoKKJxIhZjJdpRMXBjYOgCKYzQtgRyQcemkGyMXRRDzfioVgCIHgNViFtKvYKmORbvfkKWpknkzIOrmhJRoSryBHJAqnPQOkvciWDMjsqnGQCWhrrAJwFcfXBfFipNYJpCWUDCZJtAwOVdCdZkGvpkiMGyURnhUetWwTNolGhxWArkEtMmCdbMgejyPsBUOtHFFlameLpikTAunCnyVKmqwVjiBjdLtSFoIPPIKoQpMGTUfkjuaAIPXRBPjfgBdlKVJMLEsIsiZLgfFMJSonOcOLoqSlIPqBeyLNURPnqIiCKWSRUrAUcbsBovoxSgycmMMhQqDqDJuIutqORCYtjPgPzmTFjqHbksIOTQWBgogJmtBWdlpexENeOLBYusQcytGWtqshBzLFoSgoPUfuasKLvPnyQpPMEEmOvbgXGDbQrWTuuYFSEugOBUNlXdksHrLNjZcXhxUitcZmUSGJyrGuXzkWEjEQfiXqqwrFEITdbZBAMYKUWFRjnljmOCXQDXRAJanKJLjWIeWRqIbJaZrnNbqkdMFhvNdojSLitrQcUkJCKmPbHzWJHgmoDwEueueOuTrwsEkPYXONzlyjUJTclLVRljdgDfcgoOAqFYlxdHaKoYoHCkrqQFTqloptnkLGDctFpdTTjTemGNTENXujdojvdLdLJkDqzlIeqkXhaZoYWiYROHhYWtUkcUaoVJFlWpGFYnKpPwBVPtigUvVSeEvjbyzUOrPJhrXvoNSCsGTXaCWHWTWhYHbgZtFeepkBngTYjijdPoqqsOWmwCStvVOqXkspxKxkgSjUTJGDmdspaxqbpDhOXMqavlBSJjnAhzgjqSeFQgQfTNLtZWVIcHMcrpHlmjdeSyJQRJGwkAKjsgopsIIKzupnCQPQOfstVrQrhcBVfrdvQDVtnWgPCnzIvHGSxpGKjsrCXJdABFZxqVTVrJQydapqdJuIREpbhzDgheTnAVHcCUimacFlyhWSVcRtZMmOLrilPIBWwmGylnxJBBIjsFzHqejDIFIFbJSQDyGGfyntuBwkpqolvzNeBXkGlkYZWXyUPsEZABpwnyseNKqFasYniMAtsGgyEPOQMjiGNguxOwhBytATTbYaEaaKkINovzRawtijMqzSJLkaYUuHthrjNByoXSrGKjrcQiYNVXeVlYzigtxpRKHykxXWtpeaOrHnZQZoECidQzokljwIreXCgnLJKElHTbbkRCNkGpmCPCtrihKzvryLJyovxpkHKeCcVaZwkuloeUqQYnDATKRmknZVQzmDeGyGCpLLHZroMWlQZxltWrVaHhRBECqMytLKSlVspqjhMCGGiidwsVoJYCWPfVqeyDvhRtnKyGYQgBZBcoNusPBhBGWiXQhtvflMeCxABkgLKtSTXAOpReYIvziYzncrXWKpktNmfrJZHuqeRuiZJtQqYPggnPsNhcDGqNMLqbynBHEdbPQAMmXmZNDabiVBYQszaLcesqIOVVhgmkfQUtrDsAYBnqgpRmLVhmARGRpVmkWwySVhQPAlqpezfCsSCTdtcLQDiXHLDPseDVDXRkdeIHAQKzayvVAQjRpgRPkqawztCQOLCunURlyQMILKXAOxUFPmCQTAGuZxemVGCOnOeNAYpEnWGCxRjcgUCEDoOHdvZmeNiMzPLbpIHdjFIUiUvzjNsAeNApkLhRsEiyWlDVatpfeUltGeXQCImOuEsXPbmCSQRYqeFFRdBmwDLusTAKnjlbFWykepsEOVYxsdHIVxyPZyOkUXUCenkmDQapvufVfBMsQZaiXzsGmXllhDvouAzqPeIKauOmTgZoDyDBTNZTJtWEjMDwtcgmLYdZmMtpfpwARXhxhfuNRQdKiSaIMRHIXaQOHdNQCYqpPGSXLLQjVPOKTSlJeOLxSQumouQoYdIvyrmmJmyzhQFFeJlUvAjzqPArOCEUwuPSIoYYFXiaudOVcLlSfPhgrGfVxmXSFNsHuagWeySLdekmKJXYHEXLtDkZQzMFBljgfIGZQDbYUDoRblKEmfPvJBzbvzusxYhbdqNxBrvzSAVERyAuldcvZsXBAaCehFVokdtOpsSvvqVUaXDxxotkBQMQVZrfREBOczPFkHRidumDAQKnhkGVuRdmUQPGNZxNmjiwAIbFlNfkuxZJYJieNxUTEYcaOhEKcLznuORlCtLvrFcpXEGQChXTklMhqVSUAnrEzbKDLrhnZfnnnTmjofNylBeejJoWOVtOYmWlKCyTgbDgwLDNbVqEAlgzqUTNSxQvCjglPZSvVOVlyAnbRQlacgiKQLLcePwjbgOUnIpcNiUjuWbFxdzaBTcOwJysWvzblfwvNEeDCBqXXuouKDaLDojaTaErVUdUYpDAEbUouhfHbRVveAkJxIUfvcWiAaaOjHYciSzchmfhijypbvXivoICjQVDxrmFSsCBYWtxwqcZrBQPPrAHrTdkAAwQhWnZUramFLIXSLwYefBcZaGDwBBXmvNfbaCyLjlAWQgTeFUjgcHbuZaCgfVOHKeJkfFxbplNRNmvtqPEnSWgEzOtZgtvRrKfftGskmnSmLYIeAbWYPeByFHAxMmjzyrdcYQjouMtQQJKUWBqYCypJYhosmeCOBYornDwiHmVGUMpzngedzAOqQhzdeHZhlqBKkjtTpYjvGWYnJmiIQhDmLCGjPhjhqHQyhPBHeiuwqeedLAlGKVhpUjOtSUCFztBQwFZcczzXmbqVYAsgnqvAQWcuUzUNbSSRhMGYJVwxIoueqOgneyZjRINuijJDuxplkjDjFZyaimvJBXiSrpLohDCCMrXxAhqpbYTRVdsHSSuRNDdohRDlYSFjkvdETHbfncPHWCXyttBNdEuMqLplXsATqJvhltcJqwDuSxoKtHHBRfVfVCjTMDWbaoShBBpwvdpGhzqwEfTtTNAhlqSjSOAFPIuUPyFWqivsifnrbQEPKJJrOuSrZJILflQJMmlsYseEirsRQGIhyevfHkEXoJlEYAlMynFTspqTXiMBVHmXPiUdJBVPQqMoSipTyyEfnxqvsXaslZkPCUjKJWDSQNeSmhGHMuCHSLyfXPJSBBnXzHwvFPglvfRwzNNnckKoJAAWFqipvrfzynYeKotAAaPidtBWusrcWPaafaOLTwRuVjLrYslHdclLcINtBFKySfKdSNkTGlvhjHVtpKVceGVHmRXJIgXPOGparaxbrsGwHqkeCMHDaHwiBhFYuhHQKFDxcuUwehVeHSskMlixfRPzUFCgTPnHcMzeGJFiwhNbtQXOXfGxsXyNPMdwMvpchMbYFnAXwgqwiROQzzhMQkrBdYUMAqNtqAcryDJmGvSmwGWFSlLsJqzpRkcoaeGGWewJPKWWzvJDucYVlgrBEPNhitzGkdLPzsWqxqXDjbsShDbEFuBJGUNVMHSChGmGxsXYAqZfyiLALoZTcAFtcRtzmNROhdObqqCutYJmIEMULWJhKScGxOllltuTRlnWcjqKxGDNIlSDWZVekGeiGygLwssYNlymlmHbaBpbEKqcDhNBwSdTYNoYCdgtKefkZmlxJOJeFCSIwHTuFlLjvJPfSCbEXVVYBfKNkqkZCZbCpZOKXOpAABMvsrfLxjJNxPHTAMZaxMOZlxhSyDgnalSNHyZATfQybDLJwMXqnintdghswIFkgOoUyXBMrvapqruqKKcktvLhTzDAVKNOjmHrkNqOTsciBQbKJatNnQVtQPVrTiSMmKkaWwvzKhufvbSZFqaAghxrkrehMrQtiuXcIDpzSRbAmZcMmXGmvEBiSQMxtftiKYQCJRIVZoykngjReWukfBlDetIZzSPtPABHOvCkCUSuZRPVAxWjWwfnGhaXKigEsEgzdOvpszDaUZXUscRASDGjfuXKeuwXBkVIhhDTBHbkVwcsIiMGlBWlRgSatugebLzyFYPrcgSYCpYKXpHziKLUbgygdRXnhRDvWoWTwnOCBdSnnkhzjdbanoTBYIFbaLmrDMGbqZWvUXbpwzwdELUSLFaEgBKLkRoKLHnkmSuOBxgQnbmxfNYYQTEJfdhYqKdhLbeYfsDbYFLaKiRafyRSsuHnKaOJEcHZDvsAIwheooetDdVwrFtVkPBJQOhppufneFfzUMeCPrlTxzpFTzmXRpYACUtxDOIBUrxqffjxxvHMmqhRZcsStxTiCdzUbnQCLiRkftwGETDyWepOBgZxUgCnEyyZQwilytAHjYPLEeyMGwdTpqcfByuKmCMNCJDQrGAfgXdeGZqUoTbeKKcjtVkVfkoTRtHToCJHyFFUdmlsqgcSJtTOmRsSyJqLVxJjJxPQXAxhJwwIpfjaRkmMeXpvJFbaItuCkESIOHiGvooxFvxzNhefLFmiSzpxQdjbKqHPrWqXjqNOTkdcJbkxpYDsYWdMHzRSOqEoLUuLFVKcpVLDEAdOyDgNdFRdMVCOeFjLqrVLrilHJRWNFubYRWEeNpsBoILLeGzuChimtKrNwRPgrvhlgnqzloZhaItjuULKFNXXYownrKufsektfuFiQuSIDpUjOVFaHuvXVyPFYUXtvaTvkGvRuJPsCMztcJDxViHLPxQjGGOJoKaFYpOzbJphfMbtAxZewzTwidlLHFFriEkBpjEYhrAuUzdbWDDxNtPoNepzaGqCCcPlkksmkmmHUJULIpjCAZmjqjbbocNesfUkMehwsnxNEdDfyIPzUiFoOwhJDOnValUChjROXhzxFmWOTVdLqLmbkMZTNpizmsPJfLxjKMKjkUsWTGmamzTToLRqUesDXyzNKptNMYeOWHyziSZwefZBGmuEoAaUuuLQVSHChGPLjrOviniZyaqVTZhaWhdHyyxwTsnTdWDUaxdMZrGjckcwzfrLDjqLUcWwBtWMnVQwjiumUoXCyUVovkfTigkWxhyqPlFeHyGCxukaywynPQstyztvAxiUoUPkMwLJAvTiUYmsAmHhvUchoCmFjKysDcsuwykLlOCGynGaFrTHmfgNzItqNoctYhZeScJZfeKJODnxrkAfBeeHyrZWBpiSvMKZFsBPuPmstVjpjvgwfPfypIpAtLprCJJKncraDOxLPGTtJPKxpvrqEPCuuAaEygsxHetbPaNzBEWrnvbQHOneXHwVSCYadspMuoZEDfDussceKgMwBxsDNvFNGRYNUYyRkQvxjbhcBxBXPVXQYezsuPrFbxCiGaimkVNbCHbQpHiVFjNSVDRTrjYbroRukIJbfVbXtWkVyhlJtbAvxuczPXijaNGVdYYKvqGpQpmUcSoLPnycPemQgrMCJHAyOwMWbgdEdcBzDlcJHbFttjeuLvBYVucTInkkvlxAEZCXORXQhWTZQhXhrngvDuFJdvLYPCYZDRvyeaZOJaVqmCAYIcwmXXCuXcKkQFFjghTGBVPqWiarVrEvNuGcXnKEKhVzpkSIrwmuWnyYJWwrwfcwwwMhRmuxoJxZbXEJpKlMXifPEzrAJANsbwxHrMqpzcPAvEshtrIXGvdBNCBEUbywZaNRBHwxuUMEZIydMdlAiFnViARnOnpBvvdDlZSyWZQcgVsnlQMmYVZiQWiYViSTjBdEGPcEvfdoaPWIRiHpGmELebkFTILdJrELYFlXjGxOlKqshwQGHInJhiMLabOCcDjEnKkDHjJsDoNtoQCNPddfkYmoSbxHlpgvKEvMSPqIHHHaQpPYGkuVUJLebRwivzBSRYuPNMlJLWvbldFTKVDDnUTzOOrANqhHXbXVpmxEGpgjxNdslqgHuNYBqXITXMEgIncseBpslvwKkzDIOBflXHdkIvHDzCwVwggoSEWcqIfeVXHTEPIQzWIdCiaphijEiepOHmTQxgdmOguszQwKvKxlpwqIpskWEhJoIBxDsqvwTKaLzxfRqIgfIMkmzZkiRcPGWIZYVsbFtDlonSWwMSAwSLqGXTsxDVHdGlWggMMDqFFVezImmJexcKwZSmuwSBKQqAbPWrWkOnAjvnSjuCnhfItSEwqgBZRvldLXkeNFDaSGsrUqAgqlOWcHtNmrnUWsjQZOOFXsTgxzEIfxJiTecJNZbppcNdJUbUfIxOXNUdNTgolfFHXbukcmBnyingQTOEEXQcUgJITwToQAmFYhZOJOHgpdQRgbAJZtEiLFdlEUPMdSAqnpomkwVAMbsIxLQoKTNhIjUFbaCBCyionItUMHhPGdwIAFrfidZRhwYvDBeYgFQCPDOhelXZcMBDrTFfxudTheONFASnAwcSObMeQqaTvsZHPUqqyoPwinzRfeQMLhDijZlqIClptHvyBNoesDvIYKMbobhVDsexjXiDJpKdCIZqVTbpVFPWAwaVDcAINMXkhHcKbBvpmFPtIRWfIBcMDazWCXeubbxOjHzMPXYIQGsjAUkjbHEUDlBjVkZSfjNNnxrePXmiPswqBeYTjFnerDFXXkXmOOhHXWDZMtEjBiSLtrgHfCpxcvGRFgHePzUvxOhLuttbumuhggDwlgooSUojtDQdgJsDOnRxhYJKfZHOkXSOvmgHwUvhseULdfbRqaYmMEwgLbSxaogKnoJQnCyDbyckXEtLaGqLAsdGKdfDOZZuCkycoUYmRwnuZUTTHpjRHVCTBRIftdXbdAHwzTBQQetGDNSWOZyYVhwBkptvClIxfBAsFPsRqkYOMtintsiqIpnBpvmOXJTaNXLTuMqCWncntwTcSiOtQNKUzigrmmrMSsphYodgsbYstQzpGuwbWdOrBPcRikRqWjiAWBHQLgMroARQrNoCaSzLokgaFtimPbHVPutKVrXQhhJdIkzTrdEuHXuICquOMLSUpedcPWRbhRRWxJhIgziwRzjvDLlGnJKsPofhjDjBdNGRIQEaMjhVpFdxWEVBqRdtNLDnsNEeYTrxOeVLWshcVOlhAhTUqbVcwquAVgrgTtNeSoRcBLQLXsIuNFbyXglssTKBNhIrqjtQOmmFIOuZtZsIOnptSwjZIvrLHwhyqpenAPFRWpIAwlfzOZkLMxNbWsRYLTTMyMYwdsykJdErizLMpNDNkFvppgXqFLqBeWQjxLrUBrqGnDylbCqCjrxCOwOUTHaqrkjssAYsDthjIQpxIoXAMNGbQmpyXNbhijkCbNZubIXRGhdQfWmRBLjIiaELrCrvaNXORuvbYFUpJTGjFkVUbKfLeQqEmGFjZOZGlfbsRQVQdHjZHgADFAaoSJxsTPbjYhmJNdJpVarmAiVAkEUYMXNyLNleVQQjXKcArFGMZVyTzbOldHeraKtCRAfiGXiWpdjbkzbFtonIjvomRlOhpeVEDVvtthRdVWkGfnXaIslndcUuuxaqyidPiKlOKzRVGgmeeWDrJVSNKTROrsyAPiZHFCaUcqlSJLMRcaPwVggvdZUTtUvMvtjTRcXeAmHZQCMkhzrnPOJuGrjVDeIPBjwTEkzOEGLYvUTKmpnQVjvYcetvdhqnNHmyFGrMiDAgqoSiPdujlWbQHfZYiPaAXSPlBYwUTVpGPvMZHYtwmEStBiGGFGNocIeinoNHHIqFLeoPjTELRUQVTfjWptGvbwgHiEcRsQkeSzOtolhqHIfvmUuDBEINgvaZrfXJesCCGHxwZZYkzxfJikEgWrWqhGaULvsFaxYxsxVCzkXvUbrahVDTNyvrPWEHmDdDfygUXlLUADLhLADvTEYPhmPJtuFOBhNbJUQKxtoKbKjTSsGhVFldlMvWBZygXeZoAwrlxcXeFWqdpheWutLVZFKlRAWqXDFZjafbcfxYFJLpkNlqMREZCMIzuXUxISvqbzHKNPFNKHJQFQmBzcVqoqtycdSmqqEVIsqSZMRsimQeHHSHwBbeHpOoVoKjsOfXImUtgqMYzqncReoVSSFmupxsFIRJJsbwDkQCBLsAHZdvKHztvpDJLcPgJCgDxrDkkGQkljYdZnnwHhUYZglrQhpHwWmDDjEdxJQezGTIYgWKzFhjItxiLNccOMeWJlSDSAqVzQLNIMEYrmqAvndLXBOYbPzJNCTxBEPOcXWjiHtbnCVdbrkNZLhdkjwWaIUBOWbMiTOjDEErEGUSfUfHCbjmRKJtYPDXmwrGatFnAwfieozZFXOLbsasReBVbiEaGgOYOeazzwGOGnAIFsUeHBdXjAYhRIczupKpajDUvzZVEzqmNCHHRSmKljgWgwhCYkpeeknCVkPzbYWQcDkztRUddVpwqhGAkNyMsDBqSCQjZwmkovOlPWnGzLpIltCReebYzpQlepxIcYnuyLgvnVCwYhmhtBflCcpAKjwAaXldiuUGchOsPcCJoxstTEnRYSWfHbbatGkVRskpUrmfxJqlmWyQNZYLYZwwdcxTNgDqwGGrWFBkyuTCNxTyvlYaMrPaWpVclxhVEpqssZvHDYYlMpUOztcNGpZeinrAyUbCwIfJzvtRnpbvJnvHXUrDmtlBRKmImNFkSpLtnuirVvrfgDMdpVFQAXyXyDhByvHJuhSglXvIfDtQCGkPrXKHrMbpPNojmdJfKLLzFCcNqqNfTwMWPkxyABKWkbmLDJSXbRXFjYcyOoFbUfnWyDLnBUmPgWVVZxwylVSTIuMDXzJbQiWEpBTIOkmpcxsmHrxuRVrFizPjJPWRfflJMggcVCJDmKyoFdEvqjwioVcnRHXFGqkdDiBJUOWgXdtcKTYeVBIIfwtNdNAFcTjzLfeEDgfukgvKhvAOvVSbcMDYgIyOORQDVEGryvzhAYFNPvpMElMrdrpmNsDTMGvYcCKsTKCuIHSyzxWhxbfUGcEQzhtEKCAezJZmcXqOFHjDMXpIgCclNJKLzNyQJPCgSlsDWuEAXsVRlfofddJJBiqORlvQamQpvXcQAMJxSHyCIBhkQeRBnPGUpWSKpORgyKulLkzfFHJigJzdqzoACNujWbWsWXxaFxfzoOPEWPDNzYwxXWEQscwgVdwRGrjSXTotVQBnEsuaMuuquJRKJAHItTsFDtNuiipDwQWcqliQCJsNQUQMyKSJxQdctPiTotXPpXwMAneYawBvoKqGEFVEYJIbILybUZQBFWylYZZGsHgSjgLEGzQcTNfCgpdkUsPADwPAOCFgdCnPzVmXRgekrsjMCUfBqFEjoxjUnCtvWCEGZQeyYvfhXcymfSNlzsYXQHBsLwHrLBtIwMhfplEsnMDZvRyXKMPrtTRNZLuSTTikhQcQVlkKUdnQwKhJklqvqZYBhltuqFTXEtVhVFLokovpsDGLdKUsMFWdIueydfrwLsQkmWWeprIQErHWlhZGMNegmCkCuMKdciEtvvmFFAIrYbhcXrHJtFpOEYhyAiFamnHRIwSawuigpVmhpmUXWbTQjJMzFplKGbsubTwMBRpWSukrcdoxGnBuHhFvIjinCToKFdVxXEKfASnWTplekfwKYWqVBEAgRIqFoyVcLdhoZzNEtdylZoZZDKmrWToAgwIclijMcRIILDiENOGgVKdHINyApYZAPdCigSaaQAcwQqMwUoLQGgmXjYBrNogbvyCRkjIKHQyheVgksCwgMTsqFKRjHFGtIwGnQrmImioZiarybLZKXzQKxirnNerPtTMvytDgoBGoYsnmiRhYxAMvHZgkIDGWhcPHzVhIbUNnHwhxZFWLMpskJhkhtFjaFMomxcJmvhzOLESIGfXGdUFnHCgJMminxegIHmjLNgczDQqXJamDgzVlYwAECwwjVvihiDtFARSPqKFbDNmhqaEtbUCfTrrFwVvgmSwanyWXWjDCeOecmSSiIjaGQcRiVazGWqowEMGUBFkqmnnjuYjzHAkMYDhflUSIngRjHqHgMuZyeeJbqxcFDCyRhTJUNwVlGBQhSAPnaMdxfvAcovQdfBeSHhcWbwbKaCQTZBTBhaUGHGndfpaoOfJgKnurdjoyzOqvQjLxgeJSVRavcpglZmKGEhpwIYygqjpoloWtnAakRXhOhIHGxONLBpwiCVweXXfldclmIKJclnyBigMzXekLfNsuaDQHPeBjhApRJJnpaYULWKjSDOKXMOC</t>
+  </si>
+  <si>
+    <t>zqWQdoLWhLAYCwKeCiOMPeZmEMJsJvYbhjgvATxLgrCmdtDyNzhKAGqCVVqVjCvFZVAilwPfSitgRnxmvptpuTqkVJEIYmKRAUebllrVbmPTDPTgpbBPaJwPiggLsdXeqyvsTSWphgjDZAHnHQxBdBIbSKrKOnIFVwyTLLTfGVaYksALoQEHbIpnDnqPrlkAKOZAlXMIEBkjjdnFOXKFWSoSqGHGuiIbkrQChpsVUjAHAEioMWedkwUYdWCiuOAgTANujyWmzyVlwRAswEGIFkLpdCaZGnNLNLjrkoDXIJKWHeaGeXhpHgpydfTnsSxEsHJrKbifAMBqbuBPzMCUFYAYzPjJvbkXHZCMGYGlpxLZwVjYkpVbgojEhuMqmzLZQZTrxjJSCuQbXsavGLajuDKSQmeVJfvBRwZuSJOyAyipueygnSYCJWffUaeVuutEUMJGGTSiSLlLnYagSXRGrikWxrHyWlROISqryWeeoZqHWyoXctBcAKuYmPMwFmeYagHoFBEoIgDubAgpCWAJpIdqPZgcYRMaIujWrGfBhSJwRGGYJExlzvOczuZRbaftVeXOjvNUqyHUmNSAmSrLjCGEbRZriiaelfmDAKzVydyarmJBguYZOzoXqWOUIvbOGhyqGfmcrFIisXliaPwzHXzwIQBNRbJpTHkFPiPGliGHwjjDjJDhbSjSsHSXhbnVbAAmiHCoQAmSRScgeYZRAaExlvkjeEgrJRrQoTmwEljuiFXKYUPVTgjwlshKdbKwpseqZNUssSFGppFnORFVvvKryDWynLKzzJLjFiYOjHhZCsKGQFYMxnXAwHiZjoauvgYchhcrXyFriffDIeNJQTXyGbSeQDIgkdHUeRjFcdWcftnHNMDHmVdrHVyQNesFlxKOYjtLJqFEPECrQPrJjSDLPAFWcJPiJrEKQgwksKavHSvCzfditUhNNwsqqLDsrtSontwDveuqlpoeaIePrnGTdwowBgUtIJnKBpiKsfsOuTyzWVpmRcCKAfSnbELcTewpzOPhPPmyEmIsOtkMUgEIrhHBxuHghLMNLQzCpPWsXRHJZMPWMnSgWgfDntdmyPIKJeeqqpnADOMMkhpDmvyVxqkMQeGrgpByOVapxWzGPRuVFuDGwhImawjqimJGGDneLiFqBLjchteOyWwzSHIToawzUCZSdYOuhspjEYnIkEsNYxjOLHyEUQTzNYqEiglowmmChtUrtJSHUioZStSXbWHNnWcXBRoSYlrqNInMQQaQItPExsEGwUVKzJXJDmNmArISNPFqSEEeLYxEgDQwWOtCwnNeAJcOEapfffyjVvByKYCzkUQyeHKYcCiwyTHXOtorOqoMuRXUpsQzDHlkiVMHsJIUEvLGnnrwFdzJDOtVOmGxmDVfZsVMkwSbTQUbbrQHkdOYMIliCcdAQLhQbcZEjSGtpIRfDVVLVsOiUekSeWrBjCcbvyJaZXntCZepydNzOlexxdXwTHTJCiUEueTBcIXlgMAEHFZVZppaRpQPcNREDghLAlUyiPfktMSAblafYtKSZjHqMuLSQqpCHAsMrXGHCJYmiFAkRRoyacXiokpDdAspdKojpzTVnuyadxfciTfOEjzXnQmTEdenZzKRLYOydUSoCZiosblmJLgIOLcHpsValWHJDjsqrvvWjSofvEliYKJwEjrhPCgfWNgxnNeCwUdePzgNYDWyaqkNeYDDlawUiRMbeAfQRcacIVhfTsXjUARUWCDeEuNDByRnrMgUhsoKhIrdEOeuEIuEpTzZLDghGIdDRNZNOOuceMNQtcCMoNcksIUGzXvrnHeANdTTzfXumLsFZTcFdDMLWGEtsDWTOmrZPxZXQntgCquntAPMNrgGuiIqgpMwocgBjZMaCnQkIVGvlEBcmpfafweYnfizqJmVIixECibhOtpiKewppXDUgCHZbGCAUINNJyIACoejfMFMAZAQfkOqSwNBLDQFXRrdaeNugbDQuexWttjdqHeySkEKzidPbVMfsuwmQoqVYucGfzQsGFJgwQSSrmUaFwklLcSNOLbafwRMZeanxkXmzdoalwMDUSWSAgwkAnMsWQYJvcznzKkhJnxfEDjtiPmIfTUJyZYPHVvxzcYTPriUiBBRZRYdanEtXAvmqRRFLwcvLmlKEfYqxxiIHcVnNWGiTkuVmToCEmYtrlHQdGMcsabxtpFbcizYpwVZzIXWfXTielxrvtbONPhODhdTwljNVqACROojRkIYbaaEiXxPDKOzZBalFElXQGzXzPsFgdchnHoHGrTSZZDjXsomotaadpOzklqcxRGvUCzDRUtmHRUhNywIstPVGcunpYjacljJjCZuLTnzZTQQsyCKHBLBtNwzXtnubODDLdVpiMWuMkPWeUIxICekfgZfOpawrAmNPFSaPEzgQAAGlrImgSUAgKRxcfMBsKpRaxSejqucEHzKTSumKBrqchYowWJeJfnOugDBmKscQbahVDrmuCPYBqsgmUfIrDHzMkdqzyPQHvrQOzjtimsveWCjqdBMBHjRAsteDROSUmIvrnvmEtLDWtMqZVtznMgFNZlkDwrargoRVGPmPRWntzddIxRKFAUrwbHFABrLKYUnElhGRwsnDfurHJoHDsQgTjXiTeAswiTocPIRfeqXXWPDBDbAAswRMXfbXfusQQAfYcOraEgzcQwLPIaiBMidOSxxpUCCMeBQCzJaCcAqKKrqjXPiRrNhpDqrtwCRmxUcPRdKdFQCzxhQoXzyiLPvJsTfGfkyViEOKfTJlgGSULYmJeupUkBlzabNEyGjKfbLdmJIOVGenLUTINSKyHKUEkXlCOQIMAFDFOaPegyNapEEXhViyywMdIAtJFHhQwzZPBjKwLWhLrSDrcOGWogmBrUlEdvhJcfCxxQfuqiOYgBqdwndjAsOhTZjHakDmYoZEJStyhsAFWKkeVxyxDCvuCrEhpDdLwHQCCFPHpxRRdFJAqAIrLOnFNrRprUjuHawggHabHnjeQfZOCHNxTAyxuCcFcGiEJXDgJMSexTrVYKpeIiUnXyjCmcgIFSecNtBOgfZAQoctrVqXVbxmsWnHWvKROKCQNrMfoYyuFxPRubjQlUuhrXDVWGxbrXapWTtfBkgICJiUcIpuRoWmFaAIcRVIBeVyzhLlESMXiGNPBdZUfTpvkZlghSfNaOwEzHqQwJDYmaVmlcNWlqFlmDRdkhreUigmvLBCcrOqvQEnwUoNBPbCLXIdBbnsPxueyoEUImyAvCWmTteARSZIQsGCIxuhdqovPKkNApdenjlHVjgxWydPMvVKKTDOgOVhFsqOitMibSfkSQGBIaTbDRVgEsbbeMlUNCSbTnxpbzSlatnzBGUnTDuLslyDpYMYmsYaxxCbuwETZnBciSKHXkosEUiCIscmFWfkQzuxHgFioItspBIAMYQgDjoIdIUFVIyCooWEpROCRBhmZdoVPOiIjuRGxfGTRnCWAaEUkSWyXuupDHKAdQtGGHFQZDYkBKSRuHSPYrcFqsxiQXwvBzcERpktIpiHWrRSlybCpOpHoRRfypKZesrjUUYrrxTRpYdddzBUlJNHDSrswzCMXggKsujffnPuzfePXyIkuXMgISvJYtbKMaQfLDDywuJVmTDfcUCyvHCNrTHOYdUrOoazXOpOySRnOzQZInHdAKBGTyztiRzwjcwMISxvWxthapCPOJAkbMaBBVQFZqeXMAoKpXnTHgHVENjhMCTQKNDOqzkDzYlYPvzyEwqSmQlBzmTRmTQjzvaEfqjzZGORbbIuyTqltYXwTSQwwdPgdpgmgFbKOyGIRObNqYClWEOlOukJlzcKBNvDWdrukuSPtIoWMyAYnLPSdjOxQKIrBsuIkvxulAFjSJrtGWtzyhgprJvmnyOhcCusxVNDYBILDetRkgfqoYGTkgXpiInSwjdgeGOutgBbuNZLsIOXtSctCRETerddEXuqTDJjrDaOLMnfTIkdmryzoJORMcmbaAaObzaxzeKlVlyNfcitGMUkZvEAsnbmZZSNAMxUbtYIZuBkbHAFhppAQTYGMotxUuTRaQumoAlpvEJVPxtkzhAWLUGiPpDYUawANwlIRYjtzaxTJZiAoyREPnVWDttmsPuPFMEDBBJqMYAANswLTkHoeSpQkIeKwYsUyBuwIqgaKKUanPZilmYBdTUJXODsBsFsKDskfKzukuSJDgPHiNhnYiECRaXZpxGzUZYgEJAWZHwtppmrpNPmcNdMubPkcEwKjIIjDRiJnwlblWSqHangAzQLlkNcwwFXaDFjodjaunylzxjpYeGvGhgUzjRzsEnspkhhwlFSSgjKraviHxPwGflVioQbLiwJxVkOmlikbwwUNOVoxeMgkHasJuTqvMABxYGYiVOGnwvsmRerSvOhlJflvDFXVcYdpLQQkoplxzQWTDikcNJVALvWnCBVrnkklWvVzNLGShdwVLcfEymGzVdFrbvJWsFcnXWpegwQHVxrHBvzZOXtTqvDTWtYqKybkspcdwqbtZjsBVZbYLNZJGbayIiVmUnmGrVmcBdOMgxxryLLVMqTRAHbTTsuZBvuUQGhCOdNXUuwDqVKWmCxFyfeBSLhFSurQymZJyjAnUCPoxjMywLpdHMpEMBuZkEvIVOpwcKNSuRJyXendXYyWGoCqzfoLLAicumnUYeXwHpbPtbtZQgeaivrPjCvZjJwTJdyYtKyoexUwhZgeckAcurIpQqNBnQKqjkJEIJLRunAglPhPWMbILDkZAXbujlBTOslpaxRogNvOpyjBTdIMrqKBqHObkvSlImbLqkFccoovCJYYhZkdBhuXuKxWowbYESHxNcVyKwqKgbFdlMrQGjaUSQbXsnCEyPaeTIQWRLWpmLvsJYJkCWIvssxibuiJjDrSVQOVDSfxlahZYmSAwfUTBYWnMaKiLmQckpianmZyRhruxQeWHEaMLryuCZpvVlACJvieNKVBvYzUPzmNMkIWUUWoWUNKaMVJvPbtLeEeoUNjwlZbprcOKbmynOBTQJOmFfXvuHtPUxtDdbELXzospCtyZIDlZsxTXJQuaLSxNmxFwsHlcwgJSuifOalMktOcbwBrXTXDfvBPjXkRBDWWzJbAtNOfuaQTrWFxLgoVGLfuBdYJuGYBgEcanyzQXbqUeZwJqMoCFhDVbFQtjtvxCndWuoHLCmvCzqNBPslNSaLrBCqGkNOXSAPlnMidkYnStoHIrzulVYmfvPmTkBmjYAHHSKEhYBTHMRKzFIGvhuETGySCJHLaFUnRUcRXwWmwYNTKmwGcTFsUxOOCRgvuAbILdevqaXBqUlTYXpXyDASdDryyOiHjJepcPUzPiIHbxxSzJljYJZViGaMyXmkjUMFRltowcEDPoQRtuqGBGLLjveTgWbsNnRoRHoxIwTLrPpvefXXENICaBiaBcChdIIkcIorwIlkTEheMmjyFGEFYUGpHXnlBPNQoxlpMYlExhSQYBLnUqsKnzNPNBBolceMRHoFrmZhzmfTfTugdhqEiQDgBYzrHexqzObJrHrsRbjgxrpazkqCCLmwDsfDsgkshRYDLqntpwlqpnfRyLXcyUzUjteWEPEZDuBKkTECfvcolJWzdoJwkebdmQPmuzBeAtWnKMzcObsttnuQzfDOxhqZuRhPZSyIXUhPjDMsYRjaeNZmbdltGklRvttUvVpXZEXUzSMRONzOTPzFwytUJmStAmdLFIAILDfFHFNuCoZbKUpcfhDATvGtnbXLjXhEUEGBkrChiwehobPeDEsXYTWSoTunjKWVhjHdSOWXAAhJqkeHCrHWWimtsqiLClHLPvqHtScHydnMdLUGoncZMeLBUFkaGyGaPsQpdwTglIqozpllczaQVUEoezptFqmwTvVydMWlZjZxFGktuKQPQoyDybJqpPrDuVFEcByHcpHrJQQgJrCBegOhthsSbutrunZxxBtLjOJsrCUNfwPQBZSkKGUtXnjMFivolfLcngWRzNjiQheNkxWSuZJriVOcyWAWyFSLHaEDxJiNXlaVmSnhYIusdebOmZOQXJSlHtXGJugTGcLAytwcTrmoIcwmqqsIMteqYudYdsyApMdmbdAkvsQeIpwFFZhrCznelBgVyURnkCahAxrSpjmgDxXHAlchkLFqGOBAWSGJrTRmfleDaBdWajBTEMCZoIywGJqTiyINafdGNavsuuAlkwKZKzQIavrYTBjorQnFsbEPsNviXQavQjsEPVCTrGWNjSmfPmPrClyosSHNPzXQasCloITlOBdEXbMYsBcbfmDAlmsHywnxCEtMfHPbUuyDpWCLtjzbhHBfjZFrekwfuujcTJERCOyCCVJngQoxbcbNVaIXFSlrpHonLKYoEGKQoSaPZOQBMwXiYkLmbYuqNLxPusxFGFYzmvZxmYocltrYxhorcAidMQzEuBePYSoUtXqaLIJbqjGnoEgBMtTwzzDfYkjHIqlKgRUhnaSwHelYfcQhklUZNsUPLQcqjfoLcnZYCnMvIjQyswgZTnrJLibNgYsQbKrGNJoQbuTonkEWwPOSLXxPklfsLmYNFzfycQPzpdYhaWvKvwieHKsdGZTQOGREemwHlovzWRSoDkTIRdtPbWSEklXpoUqnCyUCHDarQojYLDncNxVnHskohJeENncjZjwZXJKngZfPqGqDnCURncQsGsDucUsLRAZiwiHsFwqbNCZMYNIytrdgvtqqOztTcVPfmRcjPNBfotImUBaEoixyGWOSKludeVNLXJcsMAdChOEltOEblmxUtzsmfSWhcLoVoZAPIYcNBthcPswJeRAZQXsGwfOIhDEikUGkzvqBFgFrSmhHEJEumsqXqrSktvbDDsqQAsjogVPUsTNybQIgpayKXAuOJKTyMUoiEgrOoITjILzjXmMeHWRZeQeDsyiUOWHxmIYLyrgfcYHkXWrwZQnEBaRFWnjNcjDfptAKGiVtxSFQssfwQUrnjbmBjTNnhDqOkJmRoLbqdiDCqUhXMrtmfzuMqOzFTioSZhmPvhBLIBCCZrYeimvgVxOoTsHKBvGVuOKvjzkkusPECPxzolmfMWndXJwYPRyPUSEUTpnHrvhigxmSfDJLbQzCkRhoVDWRtVcDSFJUdMCyGpkMnvymKcMycfgWvmXOMYrlkLjLjCahSXzKODYrcjNlSoqobSvCFlOGdQJLVyaHObJqTuhttiXKHmewmmRUBAamZIYDTLHOQGEvrNOCgnoIBMjzocbzKQMmhtlCLoqSzQhEriAREIaflnuHybfPlNGVDayGroDInFaxvJmKhiHffhHJAMdgUXvGavnWlmlrsbgEkxjjmqRhGYvLuzyeloZgZpxCqcsxKBwPavWhwOKPPnRPwItqGLDGLzJVYlQYKOclMOxSgRUAixTCinclXPtpIUFqfhJGdMHuIIJuBwzcOYCxZhMnQYakIXonfagiOoXkQWENaWZSwXsKfDRfzUfbCvouEWDbuQkYvWNfmGumMrhzNSsVAVjVutTYSbpHfRrhYRmlDYpmIZbjaZzCCNHQMLwzUbSePiYljPamcHaPHZyPlqqyYCmuAbgcKQLREdsxgDLTVvOBYoGKrnoyTcuwLEnhGYhqmNGhCGZsqMCQHkrjPZQiUkWNHykautgsusDtthWQKOjqtPkcOOxFvYdRiWPfvfyYKKgJPsFsXncXWCZQIYASqJEDbZRVGcGJRvpxZgwklhRxKdUMpAbAbefDWKzLEAZWUqDMAucSYyVgNNbDQMNEflcEHUDvuJFTtYkpOtJAduToIyJQdPpywCCMCEbQcoWnZVFEhnbJZkovWjAgeuHdJiKzFplONEPGrkSGtPJNlATiATNTYTWWkqZRgtZCDwKWrDrGXejqkhIdFtHlbXKXUTORPACWGgoQUwCjNSYOwzDwVLwqkFQHCLxfSXBgzOGYOsvjpPGTCcWyZZeWegaHDhLLPrUsndnbgyVnEffWqTZvczGruhufYydoChlZRMSynklyxfoRoNgKTMFkqbqTHpcLadlbpBeSRlJCMiRyzwbKtIDwJZsXOLbBpdwqanWCGfaIRZmxMyoiXTcZmQKtZtRkGJeqJQVvuOClbeAqlLFIEDiKcEAuoKWpiVLZptjVBdasrMwPnUIygqyMGWIHkrTWnLchOhjCWpKhzTviWybvMulzAnUSgmhBjHAbTPfIknXaVfuIwGyrXwflWIYDtvDMsmnArhaQCKFEyabzxHpfrojvrwjaYNqJGKIYaqHQRMPAoluteDgYXeoqHNoJkTmcCSTyZsTwpUdrecprPsqaPwyCwbXIurncrEjBOidKwxqRvYhxTaFUbjUItgJeILliYxLfieKaiDJbDFuTDsnDwDzLivZRQjeusMrZWEGMuxVaUBeAEmpRjkczMmEDcCMyFKSdgaUMdCZhrqphoKcRKsHykVMTMmzJdGvftodooazOLoUxuKfjCPDmYpYcrWfEDFJDzjZkQaHqJDFAVIMtunnzzZYNuqBWiQmWiuhZaNTSsyhFPBAGBESklSWCvmZbmNfAnZDjpFcRkXKbigcDSXChBwyxPVKXAbKmZUsrmMdzcZuXZNQehgbugRIJiLRlhjcFWkkwvDNjtfoQngCFXzWCrPGVxKliRkWDSZRlflERXGGCmJpmcGGWllEeDaVKzdmvIwNigVHEYTiZDLHgngkHiJpGsaUgOdraCENDfktySqozQnXKOkleBGDfDVKcglsEKMiMaIJNPflxpkeZzGriFDCWgveanxAtPMmGgsGscVchhzVGGIYUgNwomjcEHuKFMiSPuQqnPjLFiaiMcAcSoqqRSWPOBbmsVFdFQqhfMSzVkfLOrXqGYHgImdVKFZntPCPqmJSjuMLDNLAEEvzXvVtMqdpnFBzpBGrNlWmiXbmBiSNvPmGmyzcmnSIIEPZzkirDSHBHkDAoRUagPkkFOzlLcwcZVOHVonhRSqxVWNdcUAiSQPTwvMdCURSVXYRUAsYwuaeWkfLFnAJphREtEiHoGzNhsCquDNHEdWnmqnuqQwjzOLGyHFSHBpuMlNQiPBNiYTXnkUgwGQCrNpeTVmsSqMyLFjdnnXftrRIsJaBVkoRnMPKOTTIdjMpJYUJBAOPaDlhIsHFxslpkvbNEyIvsbnIRVyHpnAGMUDsklNMMtPskJqFcJFokwZYTeOasaSvlrINYAJqKnOLBeztmcDXptCxvJQRbjnRqmvpFqqoKWxtFeVtbfODSyjBEKZeLZGDTMhRRfIsPkEOixDjKaOqNNUSJzArjyZoYzYAIYbtkBWbWOjhitgucIzWkqDzrBlfShjgNCWnMRsKeZlsZFMeGPUKMQMcemUelBsCTYEMuWLqcGwnhFyAXiUGpuFkNxGtBASOfquoaCoujjgcUgBFERfZJTMIvHtFHvSURlWPnOvUfZpzFkUVqcecwGTHuidEDsRYevtwqWDRdxvMVIZiCaYZHvzFkPVkMGOZyuhwPGFQJmUcjJCDTXoIbhvIGgrNHnowkOUCAUlbFATojnSXjXLVqSkyBuVdABpKfDKJlgqpLzhZKIJiKcUQIFlujXqVAAlayJaQasyjwBmdMCMvSUlIBOkzawTYKgCBYUDGJJAUppsFzRyiDtVyvOrspvCjgWaamUkdlxsVRVIkebfEHDuFIwfbiHPOpGPEGoTxbAMCNhYAycOslmBRIFAZiekOigppQVYNwjzNZmtvCvGPQQPEkYtyJRNglOCajldzDujLLMEbNddVXjgFtWNbYzCiOzXGXkYkaiZIlvTassXoOYVStWhQAAoLvAIwUxnKMelQJCzciGBAQdQJtSMfpoXPcsEjIUnBgTizhWzBAcrEeLknHbrqHywiUbnjTEzNVAzSsOMYAmYmRJqaBVEGeEoHzOqlYptdIYQsDUFZcOizGWjJPAAGbdQOfkTIFShOmDBsAsagRDJEReeqvptRjzXvELmSieItejcsXVjqbAoHtUnQyBGthDxDBXSGUxjlhHJVvalafFFNKghxWulsWXnqVXZqIVTHZVgXrQUYNeYwhOlqYpnMqWiVFYaUdNXNGlJVBvIZJJgHFkcNlDciflsMKoaaQznPrXWfiiVVIloIAkkeATYENUwNSlVjBaxIXzhmxVWdfymkaaJutQLwbrgkAQOnJyPeZEWyFahxWpPKklCLXpMbEOUpfKWJSUxQbnYsMrdQjHhRPWnlAynJKRdLiCaWQUvAmEfCirsButRudOiIkdyQktCkoCVddvqRAVzVBdFLvYxRGyDEUhhEjGPeDjqqXgZGWOWtBsPQeaOpXhXlcfWJNrCuZHztBEyUIhHkLpLpajwWSQDoPYHmQXyHxFNnGogmFYwXYaEsKWtmmIkjJgfWvxlLNLJVayQlTwkgOKuppnlLmkFTJCoPRcuRPVICdCOYuCdOfrWZWuOWDvbVfFsJDsVvLwecnhmslQiDrfsBLLXTXcKgieZtcYPOjVdoWbGvUxzFtdiMmwkHxPhPohTKJDKIBawaLULHtLGmPIoGOmKMnGIRZeOcdCKJgLIyLPLwmlXVgldLUbfvGvyeKrIObccjtRGRPDcOBaGQEADdVESjXNTOqloeUegTvfVMZCNvsoqfaiaGiSdBPedpmoFaIySUdwkkBxbdHlHlrxMjigWSdBoFGryqFjnUhalqFgUuDkkvADqFvpvPsCNeCJlQwYBofvmDeEORyNfazGXlCpNcMsfipDKTnHrSLWikLeBKTFIXdGBDDBBPQgsolCuzfBoesMzhGqBEfIKwgmgLqcwcJbZHepzEiWebGjKqvzlukuXIeRBAnVZcLVIQvDPiXzfrYYUKgaVIYCUOOcEnFmmPkkBetYCrrsEUCaVoEcMsIqYtHnfwSprpFydLtlnrzDiCTyKTeVKyRacBAFbLbvCakaRjIXjfbwRNIsHrvFGhabnEnwaKCGJLFFqOkoOhQNJHBwxMegtHcspipEJsrQwzzGFiWOqNkjyWUuRzIwlUOjMRwAvXNbXfYxPJsUkuHxotUcOkDWXYWojNivkJdZcbVWUaSvUyrJaFbzzVIzdUcQRUGsIDkuddPtdeQdgLArPijqrOQmtDCfRgLBKkvJddkQCLlfqRskeIlmPTSpWsxnstheqcrcqsKsqOLjGfLpnrDokhLFzuvUnRvXxYyUoZhgdthkmViBDJUGRgAvOaoDQJtFeGqpkcwxDfCxViLbYDXmGwQHCNwqbKAeUTCjhLHRNmJoCeSWkKiFhKPjfRnkzZmjWTiSrfjXSICKZDjBBFpKMPCXwBCikhxjCmoRtNZoEKrViwfdUZKytkoHLFuUdMRyCIGQrJmMOPlrxPFWeWAWcdgtHcBPAAfevlelQUwIxQvoLpWwABfZneAIrlqvYwVyzKMPrlKZAlgxMBAgUdYQMXUnPhDVOchFafGOpmBnpbSBOPBFdZjMmRqvAwOZOtyFQTnSVoPHIZOYzQUJygeaBkUZplrmcEvEDmWwTEJAHTwfmKihknlIawvfknpkPriDBOFXiGasvyLmsLEFlxNiuKhxYkjvLzHPGCpLzxmMXfhpiTPSBAVKoOTkYjiyXPFhbtpLjtYYumZIyPULwSbikSZfWVRTQyNHQDdetreCEGDAqZrwicIEGWuFJJKNUgXyuKTfnWJloXTLWQVcTyQHjljlVbCFwSfPzWzTdTnnqfHZgNblowzTNahBHHYFtySPRdRFilwsjWyvCRNBEmakDaXFYcxAqHVjGpdAPVdpOZlQERYhJQrReyDIevYolPuvgLoKFvcFqMYmQWgcIfuNQHftcDUBjOUOSpKHUJBUDAHogWOKUVChJisxwCDaRAJiMgrQdZrzYlHmhfPdOjBDzEHDnHxFzsuRHryFmFMutYrmcQqOrkCaDtvPNekAdfqDORIqXUsPGSKVnTxcHwxSuueVASTOEbhlZLbLFMAZFZgrWsXpXemLcEzfoeCXTQOPfhhIzHVXZyOFXGapMCSEtLAhurKCBVOdSELJEZnFuKUorIoQPbdshdFpDsiQioZvZcoJiVRcDZSpvyDOcGUGTWskVXIsFsebmFkHxrGtkSqljiTslVlKJqccwPivDeLrOrvHRxKxGbhFBhZLocsehTOTBUmQlDTiJbHtIWlRmzkZhGaVORTlkBSxkPhWGbhpUWNFPRpVawQeCPyMYfhXyKbCDkbxGlSrxXFPiqeTqnHolStvhpMXdWChLadbcIDXryOyWeZtkDNEVjJOlQuGVtccyDqnmdbAUAjFDHOGupQSewrjmwBwYCqEwLBjVKjiREsPpgYRQgAxLsehDPjLTEqdLGuVSrmtNcvwbyNEFKMSyDBwztxwEeSKRYVwnHmXnoojEToetgpbxIDsvQdlhxoWwEoPaqbolixRMMIwVfaJoTXuaIFtrrHUcNWmZlKuVTgRXEcikhQMGZyhhmYPuMayHXCTgsmhGDpsewtNagMwHmaCdXFxMsdMWxOWqSCCyfhWuDCtyQLWoINAwolRtnmLyWGSGQxHsUpynJoTLXOKboaWowzfDvLMGENCcpWrIAnbpQjvTNOByDHPkaoYcoZMebstkjUOQXXvjJVQTEkVBvaronVZZzWXyyjjbdMDmcXCmdGLByUymvjVKMUXKaiLpYtyBNuhJHhCHeUkuiiPsZYVNXSDYlOuPuNsPjEdWjaizzSkXGIgyETuxgwIojqAhPurFtjAZolTpnZEoGLRtqGJtnnuhKVTprQKqfsLaqAcECdnzmnngvvIqbNFuPdopJjIomjLzosuvwppIgPOVNTPYYSJHloBbRGVjtzNAoDEjAQxfMCgDIKlQEHLIdvhIxrGecXhDKebSALadOKLVoGZlNEhBlNxXCpqIMziokZFzdzDGsiRIKnPhJOzZFsvTNCEAYPKRRfzINUqSSgzOdezTBrpUUlrHOLdxrOTsVyqmQHgyGKWLWfEfMaCIXyqiRhgjdLDLCbZHdKtflcwgRLQUGftXnUuOEDZnCmCozgiMBdFImAblySFuxwjzaIZmPHzpOzHsnwfDwtuNzlkADMgQNOIpiXYVREygayukxaqKyhnjUyiNFteIQaBvprmxjeiYSDLgDvffPHMrVrRcJjeHxNFVerwbFheUPXOPioyhFOVKnkVeKvEJMqTnssVMiazoLEbuNEjWAcmvBjOwpSDNEjbSMtMySIoKwxEaNyOiALehPXsQYDNnKyGOZkmUUDtdqZTTBFgojKhNfcXUFwKiQiZuwyFWMRKfgBsZbhqpKmeSKInpEEwUatvJZrhQEHpGxaDGGyQvCXjiMxNyliyUvIfLWhpjSrAgeMxrDuVVCsFvyQIAhasZKpwTLVTiVPiCcvIrMZQzHijDWvoAlHEtQNyrbhDczGGraXBElTlGVaahtCuZkdZVNcTnslvksaOQYrJaawWXBSkQKRdokomdnJWRRqNXgzAGhEugdngDrOEfOtREdAljNAIVJsOirRVMrlWuDomIcrHwmiVvxSNocSgYFGNVWlgksRLqUxtiPvMlmxATNjWrPkNTEWZptgfONWvCtoGPORLBKTqDnQSdFuDDdiDafbDekSBQDGqvGsCSclZGUgCZOuRNbKOfdkxFcWSPpnRMByucSAHmwKYiCmOoipyHYIYxZqhetCpTCZMciDXGIewUDxJZenLyAumBdDCxUlbYAFShZuaITUfSwHlgmdeJdObjwNDDvuOkDsymEpyfYMnQRCDaqKnYrRWZlwZpdpdzGGZMNyxiBFWunVRwUHlJTfFyiFQHsnprgSUIwglhbApyMllYwzWqWKUALBqMFLubJdwWMrUhTAGiMCgTlSxcVXXOKhbIrQlzuXhVvQtcWWNAUltuMWGnsLjHwXiKgGajypXUjYNMdHsPfYDcdoQizmUeXSRwkSbxHbXCNhtGlRmsoXWgsAUobAPYKxElqdvRcFUbpgnZwBpFHlbbXktPTKjSZoWYkYLJWoaXOBbtjEKvouVQwrGgYHOPECQpVoJRzSbcuXAHuKappdWkJyAPLeSErRMahERAQUYcmwaSczdskBYAbILXGyXoqqCpQyuNOoXidjSFPCgReaurfvxDoUcwkGgJKvLGIjJgCneGRULBcNLQqjmDkcoqbMXDQGGJsuvweSvvDVVGkvlgwBUPVSAoEIlrNMQxBQqSrurVzFucRTYalTfQjRVBpCGtDtryVHkAUnNCyHkPtgOqQmiULyXkzSGgDyWLImvxgSMkcGvbfQnbKhBCJjpqstWTdvembTauumdlRLDcOhVEYwcuHhDGMyyhIrxByDSAPbGebhJxReNnImtvXfSkpkPhdBOmlcATxOGyXfpqWoPcVfVdydqaMPlZRIQKqlNNKeWBvwVbCcZLgQKNTHtNDyTWNTpywsbnJdupOtrcKmrMYdXaeIiNYbNrHTgsaosjuJOcBFeILdhOeBZRjZYkARFcQHVijaGEsmQtSmreFjdtgntcmneKvXCUqLqwpvTgIASHsmxgBZLKstvehvcMvzHAzMdgSbBhZuggybaBoAoJIFdntjMFIozqBzRZsebYUzgYvCkYXCzbSVhSRFjcVhkdFoRRJoVHIyZfsdkYvpJcHTMALPnKQEKWduWKEgZsTmjxAfMoAofxKiDWeJpTdVXpireTxKMOHvCIEwLDaRsZBycUntvtzwJeGOFYJArrsOCBwVhHoMSqkBjFREjCBeqdqpNwdUBNEQAinHQNfWgBtnhzutsmCFqMXxRxoruaJtkNJIKNxXCCbNEptnqyiQjDAGOEcXHuyGHSPeLFwbguQdLMciLfpTiMIeqdwdtwUkuZktYpxTuAWaBeFiWquSUWHvuSnlZNIMoKpbZYupJQoWmnhJdyNlYxpjCvaEJtLHUnNbdDttWxbcuNPnSRWyrkRwIstZDekMoyZZiznaacMlVonmoLiiaeaPimYuTDegKGjmTwCLdrbxeMuqFWCNOKleWkLtDuaBSnwMdohQPuNpsVXUOadxQzkbMPGBzJFhXAYwdGASXEbCdbvnYxXUxgkDBYNFjaiVVpWzXGuFLbiTwqtqmIqasPeqhJitDscDAUiBrFMgdmRTaaGMlKhHdKSZJrbkwhTtmjoLJLPjZffrGLxlpJogHUrugIzAQgsPhRZbJOFqGPlyICxdrvWkOEPjQcVyfZiXgZhAqjFahsMYOdDbOoCsVSfVQgjVvKfFklSAgxqkIAgZluoBrNrRWvtLyBjGNnGeizFrqEbbRsMYRgRalWeTRGoloRgWpFKHymyEwLQEwhCssuxkbpEphmAxNtvvldcwGHsktSxnuOVUeHJnRrkXEBBnUSnyERzmILNrLSbzjZQUgyViuHsRdTfvAWYNXtGyzHSYFcwbknXiepVXxmTPHraofEqzLZZrjGrwzWfKJnzbHkOBzRkFhJFvFaureXUsCsyxgHNegmAzRlRjdoENTmhPVgssdYFMyUUqONiqsTbSmRlQFZMPphlaXWMNhStdWiuZvdwAwFHsKfFMOhGTOjtDOqvKUccHEgspXCjVStAxjXQJboxtTlTmYtYRUmqQwurAnyuBvXXOhghIyGBtutSrOMAwGhBpxQAqvownOKaIPZaQjeDjVFfODAKRiOYeZIuuIHboYLFUpiHGfIbZtuyVQWFZXVPVCtuVWpPjihDXXMeIDPBBArVRENylXnYaEJToiHhYtiXAxYHyiIUcwMyKobGYWfrIrAllVOUteOgthRFOAOIEDEqQDXggelqwiDJWCisTOGkwvGtrKjnleoMMQNicebfWkINkpspxPmLIbGdKBWxuXPLNFgZcCBKKDFnFjTGHmWPAGbPRZOarLRXmniBCJesjMnBOreADwpWJvYPwlHUsWmLvGiZSwuPJXFIxcMZLZNZtakUWqIxJDWTrVGHFpllgsQsSqqAvXSuPENFtNlMONAGjawQevaukPqyNYcobACqIQJYpTwJuPKzekGIBtUZAxWwAtCKNTXUJoidrSpFIHNQjEgAjFvgNalzpSGkWpDRqGKlYaZOHmCRgYWdtENsXsrqXLWrvgrHJcfyKfLfIZCgHwruEeZFTCqXCzFgJzwuWOtDXbAvsyLkfkyHQGmngaXgQVbbqaNiatQkYFdMdvnHceEeiKuivVJMISkcNuaQUwQDxFqwUSNhpHsbhvEDDuMAJWXdvlCOPBIBalRVYLfdMGphcWtHHxbelAaNGZKKXKHeETTdFthAdQqVICfAjdsoWUqHEFqiENddzWBWQKfleYpIXnoySxacBCmHWbspNfzVCxBkPsmzCjzQCKiOKzjnvCLafbYnFOGXxoqnRkzZykyKTislsrTuBPmtCqjxSNqwNsuboRZAtwnsGINaGHzkofPyRWupjtIheZSJzEwxgIsnGcOnslveaNGFLhdBBjUzVpaRaodfDcYcApAEUGgUWtQeslRJuwzBvoQHytwFoHuMzXnZntMBRRgZyLqFuNlgEkBvYGLqaBgmULqkpDNRtHvDXBeJSvkxcZNRzFOzDBISjXOBrAYxcbpUeaiSGuwirkMVxZfHxRlZijfloyORzCWrOLBpnHnfocMSPhssJSczvMdONJKqVtVcKUrHpryOVGztKTJuiIKqPdElnAuJKNVJtUoRkbYfSNVpHerkAwyGLTBqISOgbKCQFPZjDJbpXgPNEXCxxqsOLMrwRmwOQjlTBGxoGDxiUsmvaPjFRATpZeNsQnFyPxLTtATczIOhXVMaysDeuSqmdDpLkSEnUccExrgbnArikbGJXRVOjhiLykLwRxJKPGvoNaosOTKoWqdHEpCszeDlAOjpssRFDjqcZYmbysucaYUqNmjoANfwMqUPKugVRuIIvWllmXmyyzScWIpAJcnoKhTRZXbYYiqCukxsPMcelkKLMLOmdfnqozEYxIQWOqAGDyoDZPgDmyakMpfGUDdJszjJHhywlFyLUNwXwSVMmHPHeyhlKJpVYBTQZlWmcnedmaGwQfwdLGRmlsnacOnSzNWyZRSJifvSGDkucebWtaMkUCOCvUZSnDqfuVkPEqgzzplqQAIZXWHgbxgKkdeKBlSTeWoFikhxeMfbkserppVbVMNbsqhTcPOcYnskDHdgMcFrtajwMZHObPoNkpaSRpzYEikHOFSPsjfjMporGNYsikbXdTxPsTfFVKEBZEuTUDiUXvdVKvPvIOzqBFgoQOLalFRdWZThseTnCvLRPNLWcqlhRHndYvjeUbatzCURoNXVuNDveKVxseDesSsEqGonehZZIfeFzuReNsQKUikiVktnErBJFnRJkhNgMTTOCSvEEQtLwcVvKFVuGcSgNEZsPBrOOSmzBoqrYmypCrSHUGrEgjgYxjAKMsRIeWOGDuyiCECnSJuwxAdsvAhCpXvhHYJVSIGRKLlcqdQWcQjMcKMkmxwOztVjjYwQdgWDuQRbZCoUJZcEwoUBstdjJenPXHVgZWgUysStfJRDlYyuSsbqxPcaNBwurDyIKppixEAWIwnKolUCiRckfJbZmXvlyAFfOCZLQUMaJGryxDIBTdhyfslpvGpkvWXbfrBQcnbHuyjixOZRpmiOMIqdBnOTinSJLHydqFKdZgaUIMpbwwalJyTmAGiRiKUAimwhEQSPxOxzxAZdyZpfMvTlKPuJEpKDxRGHNcYMutnvyABULeLlWpAJOQlbqVtBrhpKptbZThHjHNBLKvPZnGbwQWqaHMRcGnwDmqttzyMcfozlnxbsJGbZsqCNUJOYWRdgJBSoJIcndjwfqHUUCzANLFJRYnfZtKaWkGXOANQwPDLEhnKgmWoqfJqZbkGIxdrPNmmJlaPMFuJfTlsRclSVkOAXdxAxWSjdNHkfZqHRSjhaQUgCzooEOOhPFpaSxvwEHLhDEEboLGazzWqIvYgcOykfSdctBYaLfnrqUsquNuyMlBgJyRjtqVZyTDmszHnaOhxZcUnAeOjeJQmnTIpwuvVLIxxhbDmgogIfmGRcBOzmXjogHVjduLLUyujbCsgCwjiFfklXdsaauduYTVNkpskTrLOxmDmSbVpGCqNhhCizrptieMvYnoicbAvPJaEkHXJNDMxrtswbJbDyWTISRrjaWOTQxXmRgEGhnLfaqpDNbgxTaRhvxGOwXugFTrLkWfcsfSBNMILxRkMQTnbdxyDNoAtBjfUSPAdFRGXwIOHgGavodkEtYBJqRtizlueqPBRhYYtXwoXlJLICgTHFuYnTmXHGjcMZLDYffddlIChFhQHioCmARQlGRsSuytCAFgEGShFVTIfMkqFakCcqzMHfzlKhmjXIIKBzQxhpvsaYRLRZxmccUgeHPIQBZawmwxpeheJtVrykptOPnxlDCFvyKvzpuTzFwKmKCIQmfVwsBxNCVTHcBRiINGgRdtrdSOhkkHNotIvUZSHbkQZifDRdrUTsfLPuuAgfsusPxpQFgYMEzgSYGmomjLPQwCYCZGwIoGgrnSZfvoaWfKMSpaAndmNNmIBkoRmuccfQAbgiCRszeRugQyOeIvyNJpLvDtTQxtlsPXKZcmaCxgFAebzbQKjsMnnwwRDDniomSdHmmSgdIglpmcdHyWOmdlTcDzIaMoQJtexMosEhMVklNFyffiEOrAYkWiVjvtLYKkmWprPYRVylbPEVYZHnzrFCsChVOlhNVDaEkThwitDSlRGIKWxpwMQFubeYMilVrGYBNvjFeKbhAFoHbzEwOHwbYQyZimRVNlDtwsZeqDaNiLVsgRTqTShoemhOThAsTMgEXOSTtxsfQxhVyDMivZytASYeTrNfUfFeVyDwRgdmHnnarqgJQuHNGePZIFhgJrMuGvoBDWYdIjZRPYcHKGjHgVEBnRGeIQbIdRXDUopWryWqiThIhFDfPMQpvgvUHVOgRbepmHaHZQCYwAUmgQeVMCLnSxpmSnSvgKXQhdxXJxaobkbWeNhBkavEPQBxocttHKwNbBPEzWGUcwvNGmlQrGjZSqYapgeeKqckoFUanNXGUIzhajxRgLpRwZIzAEzUxGIsKFxBamwgUFUerSABgAafWHwSWcBxGmAlbyCNTsdxdCLBFqFnGLGOzuEfSLflgQNmPNFNrkOyNfZDCulYTPoFDhzxjSpHrRaxLDoXqzgYHiMBxtsWMwQzFaXPQtfBBbdNQCPVdNsMomOJeYaRkHfGCXsEMfnqtqvFasBprkCayFPBTpynJEpsXnZxiZpErxwLyjOPRgeOUgtHeyRwPlgsPubzfJAUXMxemVhomCPdKCdNECZSzSdhNCAuZzYEpeoXsUrvyvCTrlDnjgtqbdtFSJfmauzeFFopPwhZndlkasUaUUErcxJRgosJBSNGEUtUAzfldRvhLswrPbGMEInnGRKLKoXrqXxSBOnQNIkVlMNEhrChcEUdvUzggrVbhqUKuyVhUbERSnELraMplJqleoGmYgreZGyglgAZrhZZAWzEwyiYpvvurbUdssAOvNZsYElcBsFdEZIBeyjdyqvcNkXwbQfBrRavsYvBBsoXlpgkLGKKKYDjMMqdhLbIFdJIISAwKpiDadDEvvhdYaiSvOGbWaJHrFPGJnMPzrKSkBeJMzEOwauiSeIudyUqZYHQtQKTegzxksbKoWpaPtegVsvpZSLAknPJGoyoQDVmYOTLoJIUZRLyaVdoJhjOLyTTvRHjgfOiwfwMwqjljibjroFqyyFiTmHefRkThBKbnKxikPgtiIGZNoIftlJyTERyRihkBBnEJFzEGNEELIzXtnEXIMUuGdBxWpLGBsSRmsuYbdMHXzJnMhckNvAxFRPyejhiAsrZAXGhGGEihagNOKtwqrWhAHrIlLAznsfreeHIWGtcMHnwEGdNKgfFbBWbJbUJGynOeLYSmmywWIGVjVBdbmfQBrQhhFvuhGhpzguaKtVTTYvpXvhQKjTjketkaZpjuZDthrbQRNEzBtmYrCFfyEnpahnKNzhLqMEuZLsBYrmBGuqrACXwgREbCLwYDkvOZWdSwAIokhGYyYbDuuQHefIjesPElZPVbwQzuAMVBodwjDasFADJUIBWUaFWgdeTCPmHSiwhLywjeCczGgdxdHKfdXWmZvEsDsCJcWjFjUMiieGfnzgeFticDlReNzzUuwJHSBBVSlzptmxzCTXJbdZDVRujvdSvJFFGxmHVxyyjBHoEMgKjHyWUzhYvcFletWlkwJPrDIXPjvLXHMKMplvoHlwkZhFAgeUPWVoYmZbpBPamffxQHsOCnuYduPNgYfZwUyEZOSVimpTgVlTDXKVpnpRHcqdhRlXpaKpNQPwudKAdAElRRroGPNtKDBVtqPZFtsQGaLbyUfLIigdoibLbPYpJnrrOdrMiKzDRjkhvImmtrcsjpiQvHpOAjqWuvyRRdejNbzPeBDsFAIZRMvBrJUWIPEXDpbRLqYCteOPZYXWMtXqCANCpXOAwZqzezzLXxEtFvgTyBrDtekUSOqnkJARZgskmRtjntsQhtADraLkpXkwRJLPLYzUzLrrnllfjQfqxxCvuyjsqMSjkfyJqRigDRGLePdpWaRffhehpsNSwPAVrHHWVwaAAmvmXqlzDBfGeChfPljRoZhpJlyzTPshYcHpeJZhLsifMvxWxLNcIkXgwhbpLJxsGtWpLQPTSQZvSjBNlUQjpxxQsOgkoNBARwClrtopTGNrqEpupZuFJLMKxQrGmjqwUdZZvrhwJcEskqtoOmmXxiLJTvgxktpWgdzttaqnidtLWhnXIyBBADxXloBckesoGFowMOAGBJmgXqrnGhbvDFsciwfYKzgwpSKRWImsJaFlPvkGGXvZNgUzIdFRPuBNTtgPOvdTgJwVAlZIVWzmDVCegpuXRQDroRJkiHdPfzUmfZRHpVvnVaaSbcvbMqythZwbWHACLvHuNdGBxraieqQvzdCXvADipfTLMEoYXOzlJznUVJYiFhfvEjOMRYeLkaWEbPgdinYqJSedWcwYUmlgsakTjYJqZxokOeIpkUIMPvWJwReORrVUWvUcUPwUYSQHCLPvuIzHTEZfQDQPRxkcTZjBSGZLSHbFgLBYstxFhVCUmTwbWEKyKDediqTMWkXIqjndLLLUcECgCSBFwXMqYtRjUIbLWWnTTBqqyVFjdnJtWyPrrdhpKwEwycEyZcVgvmuXVQnBKfcjceagFieHRtVqODeqezpFeFUkVApEkxICqtBIeWipNJyShlwBQFNoIRVLvKAWQnYhfZijCYDfeiTmrTIZZmJzPpHsuajZgJQlzeOUyDiGXiHIcRdxDJSCNwRLpgrKwFtusvcSIStpMZmzzNfaZdCcPCbpQSxPWMuzFICPOFPVUWpDqEQVaWYEPVuaYLOifeValwEKWIzgOXbxrauIusuVKaKKwqJxqnUiYNpaLnKFKQdfWVxBfmhLPkrTfoEGLPuTKzofiKqGnRMdkeNelTnSvHzYxhsIGuYJQbIYNeyXmmRkVKEYSnKBrREtrDhcZKaAkGTgXtvuTOEhJcwhnoTJgJkCYEdUyRZnGvdseCECOToHlWxdfccrJVkOHRLgzUhRhjUaNMFLZVZWXSZVJicKImRipYGfIoRsUZrwbjdWmgtSvjPdDOEIkJUKxCjhvxBNYAZEQQEEwnKpfnUpUEHpzaQSQXmeGIZtOkesRyhKfmLMPNGTpghXxliPJuDaLYnSIEhoGqpZGkQUbbcrHuffBjVeoIcIparqmlClhZNjdEYVmDKtNKIQfXrlTdIAEwpQqaJUpzzfXVfkYwTiTcpnaKfdxOezEPwBqemvBpVqUIDybgpApmicrxftjABpOQRbqVGGPzRZbuNaEQpKUfJsEUTpIfQlAGPdPTdbWCZJXExqgyutgALXmYLdcQoSmeFlRJZZkABokzQqiAosRCeXzuZIUirAetfrumSLiRuCGGwcgrWMZdklRXpOjbklCuatfpXvonFLUNBfdByOciFUubFSTezxTARlOTzgnIcZnobezsJxRVkPqSTNOXHnLNAZYViYGsoPtJzwngdOROPQvbbmUVXJWpHHjBuhxADAkSJMfbwhlsniNKpSjQwravtHPjgOOTKjGzCQnyWgyhiDQMFGAxYDOsRgJKvVAGHUaMqeDRuTEpiRaPLtpeZzihGBABALzynCLtrCYrlsBDiugVOaxiXYiWGMrEAYJNopIdLbxUNprZcwMYPyBdqWxyGKTyXMnOQkOURYulVIkpNbInlOlILlbbAEnizibqvsgxgwgwNUhBiXDYJLANQkOvajjFfqdfgtibpkwVtqXQTfiUCCIAEmvaYmLtftNsSWCZENoRmRmnpjiZcyzhqikCdCqdautuzBTjKTiWZdlzVzRmzWHFPhEszjvQLexltEzsGneQXBSyPvIdMDMCWVCzcRzTrDjfURTIuOImquhtrbBwyCkysaQlpxQZUlOAGoVcLbpaMXQYZDeSfMWQXpaaXtjKpDCrmwofFaznFdGSDHKgzhoAnLdezOIrXpqVHHFxKpbhUzctWsdQlaVDYNrZdhcNkvKuorIbRTiMRgzzRmQNilCLfZvTKWZjaGjXzuqmwdISICIQvcChNNQCfSxcxuUUllKYArtyeBlgFgwvttTygKUzEhNbZqKUHbSdnACwHNCTLuHQQhCcvxJfFryAYjGuAhLjlUxBWgKAOkenLaSHnNZtNXMomNvRAQXuqYUChVaMAdLrtMuJdpVxUlAqjRjgLkxONbAdfYOWBoJruZhsBUVVoqQLAvgnrSInAfZhhQzMaJAzcCoMEkuVGHZVYsaVxBXrPXjHSxmTosYvgiWergUdbWtcxjDmjniBhYQuEdtrHyPGRUHENfTvZYpldIzPmUKoQrrLHMQIwedJcGSpnNAHQXYyDbqhshxvERpQOsoLawYNlrvWJrCkujvJrIxkElgOGbIQDWBnaUIdCRzIOMucfOnsfgeEwmGdNXyIYzegFLeWEABDmoToStKiWCDdDbyYFaPDOPZCDQlXLHrhEZLphouXNHnfpKtaHXXaSXunGalwJTvSmlnnZuwhoVlhyxipTSLLCMmYxipnHUnZSBjwFIRrloAseYUfeBvRFLgGvFsTVzTlVyKLEdEbmUtbGqpuDSMsiAMNZpmARCbScLosZrbusbfFvhaJylfGchIQbGxXIrWEzykBHkwZIjMYgYBPhjqSvuPWUPFxYUFyfQcFUSmUjHXuZKYVQMDkspGJdfYihLNWraxtlrNfESPzgSmOzqFpkPRlvajxkrAYFPHbQXUJQagtGpDDIiOWhepBtfXHNzNANBUqSpuVhZKvQVpVdLevlQLMyVXmYQxxuUYTcmuqTIOVWMbIRHeMzUlpmPSuBTWBQnTfefhUHNYnNdwUdAGwZKJXXqwUVRpBLjNlkXjwbqbyZNTapiTocXfUnTvxEAYdDxqGfmtzaksYEaWhpfBTrhmgwnWCqVERIcvPQRQaaBlmukVasHhvuuBKsNdxinjjowVkTKlvUBRZpLkwVNsAaPFmjVarGbjgJryfVHJDrcMHdgGpAxIrruvHjhIdWwTngjlMFuCbhIOJBmKxgqRLJmghrFEVqCJsPtGQvnyRdcdDfdcufpCWlMOQNodRKVdthYujQzQFhzdtkeZPaNMqkMQXGjHbjCUvZgOALEnKqZuGYABLZVjawDcHbxHuzPALVPgTuUCvfIwPVhPydNFtvptFoGJvTBpuOnHJNeGRHXWWpSEnifvWwxYWTLszRZNWSQspPWcruLOPiNkwoeWGlCObFvoJUkoXbtKFpXjVoaPPiyoGeWLAUWMMuOtJXDWPJiEYVlwsAVWLntzzNZDExscQGclYLMKHWgtIULiMeUZIMFoISLgfzpkVDZEyVfYozwIUKbhOdDmAZTstXgsHOgJOiMmAqUXOuDMoNDRgRbbcOktCPyUxRKesUARgqHBlTgCyCTIjVkdeaXSWqJNgsMzXMbqhbBwUZNNnXXAxyUxdSytLjYPRWaQiUCFSjPQFVumORkvwQFBZAXmdUApMXzFngqRNAMeYxgvSSSNUYyoAyAUHXTsoNvHkNmaokAnJDKGukepNkPSevFsFtydyfVSfWPyWNNmuePjugyHouzFenBbQYTBRAojemPyfjOYOvwHpzIsPxoZIZMDoLyKweRoIdBBuqEZnvXKgDCAsQEUAZkkSBqYImlrkCuuHvPYYClkwxNXbIsTeqSyjLGMKhNTkjDsjeJctVEQJETfRscdBIuNkBcumsKVLxnjPTZihlaziziYNFHWEsgecXVcpCQKhVUMdChjViABUEPkbYnRkEDFdDUGmacaFyljRfFHTyyMJHVzXVyOWxThHOrbCndrjFTBDuXFOCGhcqgPvnCnigoWqHrxyqVHYusGNrSBobbhbZKLzUyarrezWnzdLyTkuxprljMBxSENKZtKRenVJzpGlvckauGgbdzbpealYjbfeaALYCYTNUXJHIEWkGePziGqOxsQhbzjkqcFGsDKJbSTGDAIyEBjphVpoyYyVuwxKszHGKgOgebOdBLFrlRflMffqebdgXbVpMgDmKceljlUmpqLGtdyWuYUuZAkcTLrxjvmXQjzJJgpwdTvshtisbbzGiSwPQFBUUMasZssCjrPvUpOcUOPgvXvceRGKPhfZrEHjEClExdsiHFnldRYwXoKWfRKGGLYcoWXAlDLbPQUphtdGbLxicrPSticXPGyakwyNMRNISGizFNPsLazQcMjauNSymJyoYwoCcUUusKbPQerksdMwMcgdZBpyQSxLhnuGytZlxVUqnbkUlXtiTjCZButbnJEFssTKJrUxPQByNFnNsamVYMyybENMlgORyiduABnVynZVvmBegEBOvUDxpNTShVSDChaEugSaKeIcFtEBEdkjJBcebZJawrPGKZKqPbbbBcaZrksqCMcdLcFLkrgyTKEicHTVswqpUrdLGuycfSecmhLtUAOJjVyFbfBiIpxfrvDZdyXqIIiEvmbZomYKUSYotKpEbTCbELSAETlBDCSbWdasMGqwOERoXXdSmldjqPYYesPhxaCvhCScBSXRofZGRwGQkbfahXQkdNdgCUkjdtpoQUBVRPBEKAaIKWkeTPdfEWoFTBIrbTFOmxtkcuehegzTcXovdyxSGlhXGfYYzBeqAcAUfEBPuPUqXsPsvyhEDgrkKEBcBSiMwxGDkjcLvMufrppGmIdMxjGSTznDPZRZONMXXUzYFQSocrTZGObLmEYpQSkEVsGipbAJJfDfZUBzszxXYQSkzVumopPBXXItuPtTHrVFpMwwEoZkJkZZycDcJzswPPpRwIAZwBuOqkMgfYBpVeAdGNRjdPnRiMIrJiJMDgOYOzTBTNaEVZfZNMpbXADYoKvSVVKLOhbnHNkGlwwHKxehAlairDYflPxiiRNRGEoHwhqKVPfEoKTRAoJlNKeFZfdkmyLQRcqLQvWyXCQfNdDXdmNSpEJwfdJEwMsAlLoJDSoUhrIWsvjFCnOrWvIivrjWFEfZFjrcFsJUKKJjobfdkUSnLCjPNaVyvoVcWwrlzhfLGIEFpUloJcjpZqBHcrcCBoaRmKfnyRWeDqfvWqIQxMUqSqTZSpHByurrWviyskHdWLjuiDVQATpvqNuAXkivdYnuEKDQGHFUeXKiERpcSfdCtsdJCnfhvkJBrCYAjulGudxPxDMvRtoDvkixgqEIkTNwprTMnXOsXIdTmDqgQznzhmCvWGMSUbjXBoVucWEUwRFyIEMQuolCjTxwpcqSpwlBISNIwQmxxIOPEtJexOuNpcrUGNNmbQSgNFbfhwOXEussdpNIeosbQVIGtQqbKydoKkQGivHHfpYFpgeBnHfMqRzzTRracUplJMTfDCMCAWVweQnxLgsvrRyqkmgjONJBCvTLVCeTeTcWRCpjeZelEhboWbDoyAYULLxOZzezRHAkNPntQBKiPiIGfEZyrrtnRdUdAKXFhckVAHBlOQBDQspiUrcCzuhMkBflMskxRsTFSVzlskQAwCVJqFUnKouovKPGsEcicrzfMXjOTJelGPFYbBEiXypIMtoFWMTvKXQqSOaRFqEASpdXpvJVBBPkbnahiUjBQiDmcmRAEgVzGhPNVcESLZWGCLKodrmunevFVMUBoJkCAChTouVZGbRnJqWWnKNEOpQGLOnluqTGcNDPhTsJqRDmuMLFovRdRfRfDBPJyEOBhpqHWpkpIuaLPEUFVCWyfweuUoVIFaSuaEmLXvPxBdixnoDCewCPcqmrofHwguHGyqMxQglzcclBXSBOEviWquFWoMbritIjMpPMZdIqxjnSKPnIOzilgnRCHCeFFJNKowNxEpuDOhRTutEPmVwSRMgsdEyVpVipaDQPDLqgTwuxIjRqPhmfpSgiaBAtbjTrZcZACoAPDtMOgiIdtKISunHmewLnvAHxDOvAeKDvgtfMKBGpopqMDryZFPZTWNgZEMYDwdvnWtBlMELcuTfLObotClbuJrrKYVXXRrNhfWCmWqwJFTKESYxfebMVKvQvILzfvENFYCzXYZKtPwqRVLKgaEHiYGQCTBlbHHJgTllhsuGsKwIVsBWuwGZCrYPsyixrTWEjbwxJGTiPHUvvnLtzHehlbxnqqdeZGcjRHZMbLsvpovKKnZPOBKWRoOSvwFUlvIRYkrWPHvvqClQIvzLrCEVSRpyKJqEoLOymDCBldCOCklMDOOeQnJsqlfxdXwWHttOvYTwsGAFHfuSBVhiGPmdJiygxpdFJnGNluXEbyorvrlcKuEQzRgNDFYNcbPnUarqTxmWxxqjcRMIwPtvLNntUNpZYRkbnCcTzcliALAOlzIWruPfjtyZiZXtUMIxGdKmriepekacTDRlMpLHtJoUpKRRAwGChtfSyhpztSfsWAryMotDonsTOfOGjPowOMgUkhdmPhyMrFCDxSUkHdZGlXTljJwohDRILDLUfTUIXpDgkfFeuooWwElRXNPXEvlbdxqIPlugFfrGlTSrqqqGLncrPFeWZSijfOtKUKJavLZlymdPZgBHtZzSkzaxVssBixVmniAxDRiZsKKrJiiTefIvTdhXVjVEzONvlkXyBcJsrzPlmVkrTbyHFcPklLKjijElJhaavafvbEUdFLEdKmoMtvANjKTCoqcVtnICSdCMpcrceKCiKacmBvFmMAUZqiwJbnxhWifbvweRaMDtfOCIUatnEygyuOgsgczLCTjfFbEdoptKnZduXdImobUDxlAWpXSBAXUVCFBakmCQJUtAaRtFOIpvSldGuQnrprFQelNZLZdapUFzphfpypKvFlQjRCxzLENktDHbNOFUOLjMtKrrWeCUGUVfcjTDmeCdeVXhmUtEphwHvraBlszXcNtBWboAjVoHKDkFfbhuYdPXelcABwXpFWHDWWaQyKsADZIAnsdpgdFAAkCAnoentmNfjeeIMjZrRFCfQlhcfAnCMKwcgAgmZfkDSdAtigFjBKAFwbXPkrjobIPoOqXkLAqbTCpHHNhLaePtkFYHPuVduNIQblHsHHpaqtwnwGDRHgLSoFYNusDJMnnEZAcnDrMKbFnHcymnOHHcODBsXJVPGNkkoJvGQPLilJJRYDjxbsJeQHXEGfxnlXZTsEdKQLSWktBLooxJKyItZUSPOnfQIQhCTQbfvOIFHtLsNJdcuGlBKtacycIAuVbGQMjPWRXHTEHKnItJSLtsmuGmARwiePpHxxlnSNduSShvdjPdGcdoAuFtaTSrBopXeJGLbCBcysMXSjlwLniFjpzCpMTpwPEzoTJWVqpVmGGUJAoTQIuPBjWasyHWqnalHXglIiwSXfnSpmvreUBxmuCRbuJAkaMudYIhsVKsBRAdcsvYnwkaTSFjxaaQvyogNrHoMyEggTeOVfPNgNxVofummphyHpKAXUHzbXiYXyUdiMuzEnwxDMiVXKMKmTKysDvHByrWXECaSQCPRAFUcWeOJAvIziGfMikyHcJNqdmHDybDiJYhTYeBVKSnWMmCbcCcJZoNFwhNAeMEywmwYOIMhFVKGVurnpqHaJBIdBaFhmNOfSYQFDWshuDPvdgdALWeqRAZGNNcIGvNQhNOBHPqgNGzrrRygfXSIuCZuahLEDjvMQvNHpchEsoNbTYsEzYIqZJQxQvBynXUkQIscwYxkxmIvnERYxuFauhFHeUFLdGmHTpiBbaxAnjIQlkDhjQKJitRVTbInsVMvmGQDznglMmuoSgLqVBMAJSzTumLtUsuvMgrFMnHbYEJZIcfYrVlzFvKjNhqgIyPJLyxGwokDDhPtSTcUMVpQLbPJIlLIQTaYrJRmbcyDcHcLZdAtMntwpbcfUEURGuzWPSBYYNmesWIyvJucbMGnCEOhlaMxGuSmQBmcgQjkvzRNTwqRfGAxoUNBuTdAHMewXhEgjiFjoaoACgKyJsTSyZNrIPEkUFGJkkoOVJPhCdKiyZXMMkcriJWFzFqgVaEAAgJZUBjnzZyjxMqzdhJtDHeXxjjNFiLtdXWcdPipeYursWPZsqJNNwVCULxErywTiaVNiKYdXjRzfBzrjVBwSjrJLlPqeRtzaolzXjMXSzJIoqZPcUtxPeiKQDymMmzdcCxfjwXYlOtVDFKfdPctUHPBOHoJLCwSKqFLUUnLSXYGIhAfgolcNDBPofwpvsPQozPegFknIMEeThyGJHKCPhsTXcmtaOThKeaAajDqlQGHhGJpKTyVDJrrrhZRhYxaHKbtvnIfTGgWLKKeujpcjPGDScjzyXkKrgqnRSzOSxoSwdYQoFOffJCMUnfBrzgGqLgptAAttqbxCTBAdckTlwuOTtRGeCastNNREHUXFxfngsmaZDhfoGSwaQcyzfhmpEkIfprTpIEchjsalxmatVvAMAbNwVkPCTwHTZapFskRGbTJegbHUkJhPVhAUALlwRGTZyYahPabmXDExcOLJocHOGjWmiYUafFwkpaQNbWJyfUtmHneZHiPkFuzqHiipsYntJVjCjGsqcvDeXEIecdRXGpSYWOZJaiDafnKdMWigsQythGqcspzLJlNbGkNEsacKHhJGXUtUmHfYFsXWFdnGyIhQVwfmHFCcLSYqspYVKSFNQzeiIFshHfnpewCVKgtJhGZzxZgRZgWCkgTwyaXnUDPDXGoEePJCsUhXuZDfHaUABrzjmbMlKUPIUaKOKJJotWcqADbKXqgsvMapWDRvZoHBGzXeUjQaTvtfObsNiMnSSBnfbTogAmbonRRJTMIIVGebbsavWQFNLVsVTlJlqevixJmFTWcqfMAupDquJvEIwcIWAcWbTodQPXaewqVRRkpYchUiCBsMRYMEPeWWFAOMDNJtJxaNQxXeSXKDMoeyUeliYHFNASxRrqOaUaGzjmdEeFivQXFmWekROFZCVyKiAekTOYzANABJkzvpppHCxVfQscifmdBITHQjDlwewqIMJDzvGTJcDfuaZlmxCRaeEfsZbrDXzwbDcAFQTYRpdShIPAwsWvACebqZOghlIDaCjbDyhKQeYlrFnDmbkOOnTKYqaOqtGSArkIBMCAxcqwuZxOzIkZJZkwgabatieFXjOjKKdZlyfseZSTvLRLsigYwTJFDHknuZemderBISydKDSweTBxcPWmhagAZLRCNvbozbBXPebEoOGlTnolbqzVTstEyCemImVUYJbwhQFEsyBhyXKENHEYCZgcViBeVgWttQOYQHJmTytQSvZabQjQEOgbgbJWWNQsXcXnrAzcLHFvjxoEhbcbtAFjteTFCGSBCTGlVEfArYGiKznEjarypNJVvKYtrUwAtxxaJXuGnGZnsnbBdtruFCzUMykMSYUkaojOBprDUoGkeiCPWNqkBkcnjhjeWdcNoNsJEpHnWJYLrNSfkfsVmWdBQtxUlJAtZzGJcvZFLCwdpKUThhclyfYWldVJaHjoQkDrwxdsDneCOaeyiNdkZReoMhPxhGoqbnqSzhDErgWKNVxzMEnhgRoZrtnKagybYlanzJxoZFVKqNNKNjPpyALSyTzTCZAUiJccMaZdgErQxxUOnixlsLHkVTMhdCqcpKgbbNwnHKHQYqmXGfYodCZsZtouWbhcZSgKdWHGQkdTzuCctuYezsnyYXfeWeXcKLzvEsuuMwWzTjZSrnkscSQvBnEZSVeQhxriHiBvjAXUwVxqQlIdJpOruMfJKvATQmZCdNtMMRYGSMQEnhPqfxDINckQMCfDOsiSzMwCXLenhwznZUaxmrzhhWJrnXAEayTgDhPHsPRpKauWqPvbbmHGrRQjPOgItzppxHDxxqnmvAyuZHMqVnbfyQtFfPtXsZKAKPlFFayoaPuumueTvKCJCZazWoeCKJJXYHbKKPHAYYbjVOyFSKkDkQuJjXhrjZnXPShvCyIyLtiZMIuYIPIdNPTsHXUNHAXMwsViUaYTxODIRVowQABWIJRvaKjkOXYMgUsDfBZwwYReucKbCsXcXHKpojTwJzAUcuJRjTWXMzewdBSiNOFLMBOpxtYvLeprLQNvPgSBmUHRQYmyqEZsZCrIzCeXWrgRDJORNykmUWDHPKIDLfZLgNvQAjhsaSBoMJqZargaVQsLkPutqsodYzanwEXjNIqoTHwHZFrKAiTdPOpjKWOJhbmbNOhusClyOxdgzmkpIrQwIzXGqdJqvmWtPgNosupykcJgOVsajWecSGIqyZORuTvVIvCBIjFTvoKgvWHeGGiYktaryjZHnRVPaSkxOIyCPZgGslClWRFFRrDmXFKnqkvoWztZUeRVdvZXvPCYXaMJHsKbvLAquSfpNsaHAbStNZoDNeQhfnjEpIelVKsiUREoxWhoznSYHjjiNxxlzsPnvsYvRcQlsSoYkQokLEPSDHvKryYDMYfnloEPWZITLKoxoztaOyRaZREZSeUJBAExVQvrjzFfUkKsxwswmZdkVUAOzXhXIJOSmEyxeKLmXqPKmJbMyLpRCFWETIinLnEammUIJAsblwUwJYuIiZXfPqQaPHhdZDTzVnCCuSrytRkIytzHNlKCKAXqmltpIatwxkGCKEgLNQakMsNibYRrUEZwwXOaXmSvxvqAZltkIhNXFfIIMLtwLqpKKeIWrPjswMJBFLWCJhEUponVfrzrckZduaBVauHItISLKXRBPeHNwdIWdOVmWARwQNLGhDerDSkFRadzYhIQREjlDgaVKOxNEuKGKnXZAYmOvnCoekkOQeKWggcRugxsQFLFCjCyjpPySeETcKsMRHNZypDqyzMalCipQlVLAGFIlpjVRXNcZmVJKZtzVcJzgZNaPlsNwGADJiiwITQeytPgeLrYmdspyefJdTsFuFFwIkTEdKutMJNpJtklVpGZORVKUNPXmOZAmPvAIOoMSFPhqcVQIXYuvuziurSgksbTlQxDMyxXXjvjmiUgmRvUBAnfTIoAOADoWziRsVZvuiFXLMMXogCfEaNYlpZlPtTaWRdnYTRyZWgdaFDTTNKLbyiVdYqcKcbbDrDlsqChshpxnIBLjcRkyMwnXFEQCNIVbZDMnpCJjeaHFQcaFUzpwNGVjFdJBsHJGqmbfMvtuFzDAnknmMtvxOMYyMcrkjBhfxRWsQSMJoYqwcClgcIrPttYPLsQNvBlVSLEfZyYYSTIkQOFqqenYPAWQtewJVzMkatwXzROIQAscUCklbGyLlmJnbyHwgYjczBBasAWaKfHLBIIcuqTCoiXNVQjQehfsFxMFrvjQBqDZbVGsvFEKnOfmEVLNuQxrcJdzvxyWpMvOFfIAnfyeueYgcQudsyJrCKzXvqCHeHYoCnJwlnraDtavSerLAUCnoevqVXcqZwKCrCRrpvzFynRvdffFxWMiYHiyaShVFJHvyMMFOOSbqoYYaRZAeOXCdpQqOvoJCQwCfKTEttzMDvnfLwayBQXgXzaMmwdfYxrQZXCiSvpmbAXTyttgQMIYgUueQoudGdqUhDdgmYUZFedZzmIIwrqPLLvyEiVKULCCCKQciOcJVVIZvNnRUTjWXJHvUhtNqLTjRruOVpEFpUecYNyowPuifWveaLsFXAqCDFcSAGJozoSNOspKxZYoUZsCDFQRXqIbxnBdElCpYncywvObERmIZufeuOXdTMdDBGqcQvJbUBkfmPiaFbbkDhPBWqTEiAbagfqkzgoNLrLFDnLuLijjayFLYPkNYwnBMPbZGPwnGOkJuymDYtjxTTKMuHfCtRHjzCeGCulCUdEPzwnnxIFiiUxLmzUiTXoAxKHsEJFljKwaYweHLgsfxnynLatktBEwlwlYbRpbSjXGQjfnzuwdiQlbfxJSyZcJBlkOBpEAIoxclOZTcZRCEbDtIWFeNcTJZTauZsTmWYmcjrOuBzpRogbOUGWifJWtGmBALPaDYAjGHuZTNDFHcanqzNiTtfidiRrJJqLLiJXuStPpsJROuEepYAGrqDAFUAVtwOKZfyjmslTRVNwDviAMUoXtTYozTmhosznJqYhObaZAwpDPJSksCHZvrmahqrHTyslZsqShmORLAuUciAvcnuegCmNHBpXxpeRLmMeJsARPyufIkimGAQKCstNaelxUbzKxNcPRFIkAyJAYCnctSjMoRIrdDwYEiXBUrMEcljkLeibcAUyJsUodnJPnyCENRNRbvQWUHFgWxHqzyTAeUrJcmAbuofxnxdxodZzZJiSbqcuygmnysPJFLYmLasofFtvEnfGpcJBwawGPLvCkAJywKknwcpvRtrOLGTSxjothbALPuhTaUyHQsjwlgabFLBQPFuyODmHfhMkeDjQUrSQHUwgcOnAssVceHCmOraNDPoFeEwlrWNItupCNbGQClWfGMvCGlmqHZlTWGGzUzDYSXpESfuHTieuqGvaVaWwktmRXRgCbeIRcLbKQLNoHosYWNMBqxjliHsGyczJdDplhGOJEqsHHws</t>
   </si>
   <si>
     <t>2026-09-04</t>
   </si>
   <si>
-    <t>23:25:34</t>
-  </si>
-  <si>
-    <t>2026-09-04 23:25:37</t>
+    <t>23:42:27</t>
+  </si>
+  <si>
+    <t>2026-09-04 23:42:30</t>
   </si>
   <si>
     <t>{"key":"value3"}</t>
@@ -455,49 +443,49 @@
     <t>&lt;root&gt;&lt;key&gt;value3&lt;/key&gt;&lt;/root&gt;</t>
   </si>
   <si>
-    <t>9223372036854775803</t>
-  </si>
-  <si>
-    <t>zI</t>
-  </si>
-  <si>
-    <t>UT</t>
-  </si>
-  <si>
-    <t>dS</t>
-  </si>
-  <si>
-    <t>Lz</t>
-  </si>
-  <si>
-    <t>SLCmHwXgtXMyGSNRcNIWLgAUpNyPhvqfwHnwQDViMpUXJcmbBTYjMcmRntlAyrWhmDLtmrhyFvUGKjWXIZeqIUssWvcoAtWFyBBxpsiMQbZVxrpaDgCrJqvzMtNOOExycGCyMRJxA</t>
-  </si>
-  <si>
-    <t>HwSsyPzSCYzzNixVKnrZPjNNLbcVqLCalGFUotmDqGcRaBgcMNkMhwdvMCMXFtILDlUtKjUelKicllXIaVHmLwjNkgzQdGGAXELIQNLxbPvVrCNBGAaLpZotWWmQMIypkUMOrCOecRcAzVRPCtnVWDi</t>
-  </si>
-  <si>
-    <t>OEJbEqCxlOIEyiOGZjnzDmnIkPrLCxFjSYLiwtCaANChjjMvhvKkkIlWxQpQHtiJVketdkxXSQeRvEopxgebcZyeunYzEhdcUPwecVvtQEzcAtpanwbMSgRGuCoZgbbuShSjlkTTfGThsQaZApRvtrNnigLdefJujxOpEbboppScyKugPfbuQTGiLdYDC</t>
-  </si>
-  <si>
-    <t>oEGbuFiahHAtmzsJDhkGebnkjiyyLbEkKTuTAszxaZwLUfRWItMPzqsLzozSPSQxqtsgEKEZeRXarSnAirJDGwblefmulQWnkzKKFnSidGkLcwkYyOziQpWIURcJDWBeNsqdEYatUehviYMQNzAsyKsoXAjOllpSnCpbJCofcvFGWjFBNSlWXTiLDvRnOOpWeEmBmNXsyiVGpFZEPyratCncHlnWfxkoYaAUVAbNgrjpxuVqcpQupfvUPjYLQGQJIxXBAOmpCCJMJWfjKLUbAyRxsRUVgpkQQAGxIPIRmilquFbfkGzBHpjldGDBxhIjSmbzXIKLJzqdyufFWXJrKckmvyvIsLJQDVwGdypIJrmvoLIFonUnsRteKnsyLXsNihTZXytfEvQLKvigYdAFFpjapSotLhhxXHBsSJOJzrHLXcgTRZFmMEjxGvenVzajKDaxuZqRBKkbPGZwRCMzCdUcAarAofPOspqsVXiExQAPRDHMkTAQCzBaCNMbTiangnybEmxFkxtfDyLrNivIxmQbSJRIEXujAJnShDunKEVfhYZGBKNwByunZzugMZTrXSgzWvgpkaCWaQmtPMsBNZBFkWCivgHKIQHcZMioXEmCEInKKlibUaUoWnIwlMmoSBulijmHjdnVgLTCVgnPaUEoibjDYgnHdZdaRuJdCUVsLkFAezuLFTBoAAnlSCCivGokKZIXdjiYMxcgiUjHIMyrPHuYXdlCFZALyjbKiNvNDngqRDMoNakyYhIxHiVchTbsxyFADJAXrLciaxGVtClIYAOlaRSdalInHsrOXyJNnokWfLvYgVrxmovqKxLXFARFFEqwfWZXBFwtpMowSLZAVcPbDxCRoDjGskfTcqtOQZtnCPSexLrnfawCscyXNweDwMRcfHQAxCxcxGqMnWsimMGYpysdOGDenoFDJZAThzgYgdtheMGPIDGPirygSpOagzxEZGxgoebVWkyuqtofSvPgqxpeoxHNcTAUvZJfyiqluwBzRcldGMVqAGJmSQTRCCDhppoPTGQazbrScInVOCvHMXVoWUHTDldcjCIePMJVUcExaHQaOCvzeQNAQXiVnjSAbGWztshdrCVVhcXEssZiaOlBFSyjMJiRsRhMVSEEkJZyYQEvvTMbTyRnWQoVDdyFaVnqXGNUHEOsjfyKhfIWJCWFpQMOujFSWxeMPOgnUknrpYRBkfoWTzeXUiVCbRBLNXoERlxitwgRNJuRIgIKbRfJegVAXRevYZwYBmdzMWlIYjNgpctVYZIEEHoCNQfUBbIPPPOpEQxqUxsFPgkzIKqiBOVMGRQLfLDYXtkrXUqDrmZqBtlWNBbxTpaTBUhiVmNKyBBEvKDvfzfxifBwRrSCbvgudaDxUBtsvrdlrkeucyknErnygorsSGcEzOfzbcWrcUIcwgMyFdwecgcIwBVYhsWGPckpwOdRbPApszXvgycVKgaRfJkZtrlxJKJQQtLPFjQUIYeSuRTiLuZPWziBaKrPzHnNlerIrEsAIrUcUooqvVJAQZOtJZRhaDEWBIeRVkEHHCIETchcWJtUIltEbKhQnVaTmGBuSltndEotuCrlgSPwBuETnvaEuGPJucdUXwwtNstOGgelJaSOdqutIcFZrbhSAGZkUJZgqDNDXMXBxDJzvJtXuapZpgqYIuOnnVuQgkfjmpTqAuSjXWnjFQuDdLDpwMiozCvsQCrCmMVUgzmBqEoOHjUkEoNnMpOFqfSdVUwnvGZJMlOlWFJxzAUgcHITWFmkxnpWDrdNCvXaPlpwFMYjPTGOFnruyDjwubPlzgCxEehQlOJPTyhJJVAWkmIKHoiiQAiRNZYmIycbVXdLNFovZuIeEXitXdLoUJlCMQMwsohfmUMDaPyWKlmSfrJbgdsaWHSLjfiFrBxmaVjRDFdmgCRvGaDuPIapvxhIIZLgRKYiIeCwouxlOzecVHDOrvRssoCgykzSguHEssVNLPavoXZiGPKxFqXIGZuMSRJETopBXHWBftShoYlVshrhZsKCsUscevufPKwMrIuhmkgAMeEuVgCGDvrmLuAiMbACRYaAInrnhRnkpXsmQBePcvfAIfKqWcdEqNoYsGFWySVLKtRgPurGtReReAGFwRcFiKZTxdoFwjjqyjdIQbrmNwwQjWacpUAOAVpOWGklmUfjOZunRrqTYvRNHONjykLyoZhCHFthtUTmALbnMSMFLeeGsdIvIsbIvRMYUsbMRgmydFypSXQdzStunGoYhRIXlJWokcKcNfOKosfQNtSBMJOAxlOHjcaMDEjNJEDMDBMteraROgmCLPmeuBcIuyiuAmEFTWuMqcwjdzwyNJbSQptVnVxwqHWUsUFuJHABbLiRAddORWYaJsFhPEqmDBcTUTVnoEIPUQFdVesEEtFhZJjHKbpSCmUuPTbUNfoMcHPlZGjSiVDdBgDIIrtlCTMcqrwJMeKLXKNgxGQZHTJcJNoyVVpUBMqAzsAqLbEmkjFsPbydHLirQxWyHGokYXvtbYpHElsRADlDplOiYbgIhMAzDLsrQuNqhYPkzOmLNtPfGCIQXCCgDnThHeXlXHtyCCxzYhLnwdoVujsVMRJSgNcGaMYdHHLoCWceEmhmkCFzHDDFLzVegECiQVyPIlrXzpFFiodAHvYkrijVzqmMAnsetbJVkyvtSABCkxBqXUzhJHIgxWPBAMsnfOuMHfxhUgorEbuNYXLnqjvoWNziOxFUCoFJIgGFInMWEfpKwviECzlsyQYIFGcsbSFfyctzZfEVkaQycsybYvppbWpHOdWRwRPkkGrJGoTjegXRtyWTmozIdSeeAnwlVLAqEXgivhzdggeXDStslPIkrzYHkDdeBIhAJXnXokFYWHNufZxUCiDAKPEtibtWdeZtUKzWHNOpRkLBpfAuIxckxDocHtTLbLEuJOhWuUdbVBEHsTMsyeVjHSCJNtDXdVBgoXmfvLcETfwzAHCioehbpIVloaCdlTvQNvHsCiQMOENqINpoiFGJLuRIQUfizEVNSiihrzXIjbUsSbGUbKMVuYjnfJdzQUOxOqxKtpWXWEoCrHvJbSsMXIPMEQJLLyaZAftjtlPLgMdnFAjgpwxYOLbsZdtvVADFflsZJSvOHYbEZEMZRAcoXirfzkapJCSnFtfDcyHMjcRclbxArlxFXEJnbCmNEIykAtlAzLxrAWaNnbCTbiQriylmtDcViVUjuwtegxZCMvCfAmIhRWfuJFqPOHZnzdNyRhwKadnQnnxNnKNyrOdtsDxHxGcHKKdJqFjrkRrqnGjqtWdCyhYtakUElruFCnJTUFSFnAUWXNDkFdniOYLNHiTrzNYMKGBXUXOPkqUxDoWflflupCyXmJFRNTClwJmJlqaSquXTRcNGyuVmlldllugofocABFPBOcfuTMIcacMfYEquuxpbifwJESoptRwjvdpdAKXewgucMAYjyXFuMQLmQPrEZZvSRWBxxMPQsZpCBxkexJLNVkAIjqPRqNiczlTeINxPsxxDMrckwFeEszLumropVmnkUjKVPqdicMIbiHKfFqGVrQcBaloqNDnLbwsaGaGwRXcAKcKEkmomqGOrYDAdIXnikYsDQCrUUSpJzWMjkhyNKgrRBFMBmhiEMvBJfAMUjGmwTRAmQXZgGqUUphirzVywZZGoxTJhrkafQAaHMuihKLzqMevyHpkMlsKyvuEtPmXUqhGckhTTWkfiAQKMNipUYRibrrKIjevdHQoWLHTWpmODJaRidpIRdHXULMejFgfegyHgFqAyFqqzEkwjWsPwXohvuYockzaskgXAxtMvjQrjFbCxWkAoIWtNgPsZbcofcmLwNlXOeOdQJrvahgUfNinvwGOuAMeMJnjFABBmecTBLyGAxaGRPwNAcbWMGgBkTjzrnfAuIjthAgmJFUbFaKLkBBeXGIgyEvrtAAlvbjGJXQPlpyfzTnhUHGyljQCDYAbdnrmIHGioqUOLSOoMRLQmptmxBoyPCRbYLCtbvwDXdURSMlsKhvMuMzLLzQswrMpMvnwSPNVUQEfbdhnEFWDbDfUuQyWOfYaOEnimcIIBwbyzbLUnXDugvCCiKNapdKYvJAqcgtzlhbmVGghdbPVzTzCDNRJPeJraMhMBTpcrjKZbmjJlELsNKfralREPSUrnPBuspDQaiEPGxlsvtwCJGPAQmeCNDlSbcqMyCwZGpDAweaHKfMIXWOrgvXXHfLlcLlPQMCgoMCiZODrGZjBhVLhHVFPiNzSYRQaGIAMFhlxEnvOXuJVFLkEypzRjWragTwqxppQlINaKhPPZvwoAlFITRMnHFMHbicBLEwugThkGiKWgXEOvwWfcXMNfifIagQZoRlICdFiKGMfAvFVBIwazdLRwsnXPhYXLGVtCsObZcJCslySFPPXfKCelCrumTBJMaonzZvaSMpORvLjvikpqNlGhApQwlQURLgNjoUQGToGUZHHrebgAcGIprbINlKrQyKQRQOwaiQCOIcMsDfFSkNBrBUNhJacZNWzkNcpvAKaCGPSEZfAKqKMyGKHpjhpPWGvofwJlAFXimixWeSMBuSByXJfLHBLgpjLTVZdsQOcUilJdTNyUsfIgsnPZqMVTUINYWWXCMOPwKlwfegYefTDwfTHZQvgJuJKoXiThOwmCbUVhDKBGRfZkZIXmdYzDzQGOacpdTXNjgWhQvJSnbAPvduyAqMSVZHBWdtsXzFOBSOAwhvjQoRwCUMitplJvUqKaAxfbosoJqCsJqnWYUHBjLJUlNrAlvaitvoRlmYimpgDlFXWuKyohhZblkoWneMKjfUtyOlyDwrxEIbUNIBNqMALJnXzvMxpxiltcjUbBtSveDDgsIsJimTHnBdrkcHEFoGqQyMXPsEYWaWdQqPvMWpDVEGtfirkinHTSlmkjVhDGJOjveNrCaAlURExKapKnMcTmzzgypfDKMuTMpCeggWAayHjiFCExdKmcXxmsMNjfjYBqZZRiHJZsVCjCUhyTyNgYVXcqKBDAOaBwvICGNwpwUoWbfmdBMKhuWfVTWOBKsLzpZldaekvMMGImONeXRwvpFubiQLufXPLEoYqaPMZEQgtUWThACMQvTohdrQysRBtPAMTmJLWbxtGFrSSXqaObdaAyeqxrHtCYJHsYKMIQFYoYBmpbsviVOsgEGKPqNhUTYoHRVIPkjSfhJupgdacIkasAOPRLpXxZMuVIKqCCPjrffkooUkdltZIAQGVlDeqDHSWEDWJUGneZEpHJeFzpuKkVFdkUZLKNmEQhJcpglKqVrdonHKZFbGYBhHrYCsDTJBuXbLpQtnNcLscBqsHhCPXeRsAYPPmPpyePsRKRCQZScGaXBoptduHIUHcuWGPYROYCSrJUedcAbkHTgTqOihwPeNSjWQvamZmGgeuXXbRznXHZNhZxDhPAAkpjTrGfDhhhtZiMgihidJiRdFRUcQDMqUXKuBPoYTsNZWTbgDmENjPTkQYhvttgcGlDgWtPSFDatoIilZQEBtVqWWzOgITGlmxOcJqZMuTkGxDOrhEvumkSPMGvAvJGOwTsBdngVpMHoFRbXpEEyTThRwUpujzczObKqljLYWEnzFMtJTxSJTqLCkZMAHQxNIBHPofvjOAkLkVjfEMcqabFSfiRvFesVsAFXcVTcXOoUWhslhcxzzONxiDbQjdDiZCnVIGMHfYxlievQLVFEStSRIZxSHlsssXzuxOHGobOSImLKRRDnNlkuebWXMXGEMZQjUeCtpKrfDjNxalojrGoUlireFeXYgSaSzMSINvBlmuIoJnIABMxTLaueqmzXzXEsHBanJeOXmbYUfbncHsjoquMmIFfMKLjBCbbWDxbuoXqfIPNzWRFWFFBRMoQSyEKrdwTaqNMcnEkapRCqlXFfZsikWlsXQKrJcVZyDFPXPALPBlHNbiPQYinpCtyxuiYDfRtmSIQjfCoCQdMBNqCMrgsYeljWzguHLGxhaFvquBBisqESadaYrzcjwunBiwwiZywVIlBrgMNCjdfRRKARkkLLdZfFIXHMgXeGZcQJkllBHlKcRuYQyKipFrtnREbGNXlwUVhcsxwSfAjpxVwKByfaNrOdyrTHVNtlwdLAdEXTpdRfdQnUOPdnnUYZyOrsrWraLYokryWKgrazJlRgOXAFgUcOvzVXfHYXEfuKmSoPQPprNPjlrAWYvFPVjjStjokOQQHRTmAWXfrorEfXOdRgZtkDLABWVuLbXnlJdWgyIbvraFIoVxeczrOyseNCTiEFfYAJvtymFLTIfKCjXTfPZJuCEexyipvFzbfYAdFYvAYgRuKjwkoWJpBKDgIbmEkGybEXzRvglQVwXjbHQQTXRqZIpBtlZiJZkPPmuDwOAXwBfMjjzeKCgwuRQqCFXWzCKlFtiSOgeFQsXCNvLfvPgcxaDZpBFJtnsipGacECnrGmWNYVUobnhXLNbBcGOZFZXoPHLlHymOxJaVxqKrzFzZyObkKnkLXEUYjQutfwbedocIRKBxosoNgVdgMCHHNeeALcMMsYBCcoPMzKZSIhUbnbioQpigAqXcPPqgibdCZQnCOUULiADNBXLEAzyoqkYMoChqjaBOsuCanGWlcLVRRoCKGNokIefzEGKHmHeuNKPWJbHRzieoFzbVoKmARINfokkXZQMwdFfBnwWEpQoGFvvYSWqeRLlxePCOGKWpgZHdFHxgncCKhtVMqjGISqVsVbbCPXfZTwmFkwrDwcXQCQyEfUovkBCidhQMhIvVTGiirztajzCYzMOiDhcfzTBPxzkNTqmDwusGOzLjAFnDeOddLNUhhiCvoCeCCXDjTpdKexvgPhITONcRUpzCEnijTBDgKZsuMFeajeXOLFJdMqqaVttGlhlgqIhVPgZQLTbcFbADlRIyaZjgzTqPmomGnYuEjqRmOjbiWNnUxYAQtVuXhEthXrUkjiOtcjdoFAPNzqkFPFDMDAjzEqRbXlujRANCYUBcIvemspwdzyuzPICEJPiTObZozACjOilIEhwrVkRhobuFhyorciRBEelratsdfYQVdOwtFAAGwUUNXsFQPHoHaDgYJUDsrsgfpeqXzcapSrtuIvgQdEHkTCBWYmSEHVEBUzIrDgLZVQAWvTPXPVZSgVCQWxkNmVWFJfKdzvuplXeQToHkUWzqwwPIYDciaekWKDAfYofAhUZMMkrhjPQIEuaVKxjpSfQZLVYNssONnNTrifmpPrDJppAhGuvIRZYwrGKiGjfoGDRNowmtIRvLeMHrdkZHyIBEfBHhotFTULnwRtnKtVXhmFOsLFOlISogRQaGeAQqdWsdJZrmybycsgDNoxKuScaWvqGxNJkcbhnwqSeQluiDAWZTQSErRopQovVPgztgMGoSOkMjQqQaBSIARjNQaSznGogZjBntTokUuOucBUohhZjbLyzsXvJHoyofzJTmHIpKbKJptGZmlhQcLntJnBXMERlNOKbWSRpIeQiyqcydQTLLmbjaVstCGalPDqDVWXecETCmWwOvatsaCSvfhEmayykEwTOcLMhRdtmiOETTsYSALZkJEjcacMklIgDoqgCKaHKSVzOXrUBLraqBKzJjLjmrJQxeWJkKPGqAGvzCbrUXJBHeflEjGhsWxdjXiUIclqUByJaUUCjrvWsjWhrIAEtQySexplfhqPvWTJVhChacMiQCgKTTlSCsphPSqRsZUmvqCZRvFDEsBwzMrccjejQpJywVzILxmMyhDDNhGNUgSLIkVIzRSwlCVylXmLYNFEsFFrEleoOvWoYRymyaAVXhNqShiqpplATvLTBGzkrDupYeUjYEETBUhaJnmgivkYLWmGhNyJiajmUeaBKHZEauOHHxGYBYAMWzpIqzPamsJIOfkvzEaXrbNWCnOUlHiHCtPXYHHcgyCzRJPRWuKxbuJtNwFPAxuwBBCetgbvrPhaoilRghMkRSwzUEROwkwQUCWsNAyjmmgpVApMJGLlakqXGIITtJSyOSMdfCMtZThLcyEEAykvSLSiNvahPAkWepzlBUJlgfzaKFNlEuNCeKciTTvbjRpUwUwnkbYWCKOsEztnXAcbEnjTAkeYTeZugYKdWzLATVJrTcySXNFteSWJYENPszuUjrIEIHLXfQacVNZRAfpAklTdmrtMQmmtauahLCBfczndIWWZjYGOLQJQCvLOnBYnxHHFVhswvVwubYyAlcMkYSAYJcojXnDubOHCNQOjrUlLxnBwHHhGesADMuWctwmXfLHgmdcHsLcPOeePyTDLpftIQbLsdXcMToEFgtSujcQUvsrrfnhuOvxoBQBcPCubbMHsyzepSbRnQJQkozcYtwlDTpFgtAIxmnEPbCIYrnBQicZigvPcEdxTVzNaOESqJBmpHoIgCXfkgmHmqvfwqFgfDbBuyPbiMguaRIGusMfDNbMuXFzUuWMJCWGjThmqYaJUdFgroYGAMAGUDyvtrOfpFRhyIDJApYFnXgkmpStqoPqXvkXynrwRuNgaRwKxarnDAOUUEjIHUyCGVGnIsPEdSMWtxWbHqEblOukWOTJiaBSTydQodjNzoMiYsvkMeuobwRGRoupDpdXHTuHddBocFOQDADwwPIoQMrBdHWFeYFJmCBuvzrAZzxtwAywaqpZKLSXuoPJNcGaSpZTOuBgUXJCxEfjniwIMfdEXlbEpgXhAauVNiPnqoZIPGJwTnTqWdkXmrBLXbpKGmwNhUAfQEREHtsWIXvAogdPSYxufdQsfTFSzDbFFfbrJvsjahAEWdRDDnqTPfbxHeCWmYDjvZoSQxsSvOZDJMeLbColsekblmUxUDsbSMlWKOPDZlnOKBqLZibTpOQBXNBpYDgPKfVbdCIOLoYMQpXDTwuMybDfqApYZGMxTIZiWELctkNFllsGDgEztlyGGFJXlSkUvQcrSWxvabduRpABpYIbwmXVdZTCovcKKcKCNSIWqcTJBvfdUbjLgevAFQXbyplIuXdoFuPhKkqriwuayzErqHcRMOPaztGpjlkDoXhTUZXXblZgxAfROqZrwagmectLiOhScMWNDUbSIhJiNMrSuyfrGVgUPVPspomfIzZKJDRZFGcsOQbstjZsOhLqkqZAOYMYtuxQCoHcKAeLuZueloCaZoObmzylZSYbetafnLWXeNFQFIQUuFVCLygPfePDlkkHWgYbWNzuuwEfveKiqotyKAmmghUUFFLlXONsvbmIpoJrdnxFHGvbsFCcscGJgyJTFryfFFRlmdGStpIiKSnrsIWrnXHedrTJRCLQAtDyYQzoNNDJZogXglzjkRYkAYcqyxItVUHFZZxhtNxSReXkRiIdYaNKgRNoOeKxylUDVBDHtwDnfNlCutYfDOAVRWRlazxRRHQWcWUJdpPmFXVdBbVeDplKYSWqtJaInxcSqLZXLymONsNLoSDmkbHgZaezJtAFFVtEOkzCgCotZHGyJecQzgRZjJJkDigmlfkAxIHGsrSEQVNeWiUgzNnZhyDOREDSGLgltjygDLdgLeMROWihighcXNTpYEalePwIBrQYZxySPoAfrMZMHiZlbmwEiBdKSskPKCSufSqqYrFVMpiDwUkMSNSVbIwcFhBcbpCZefKHLjVpbmMdvAhYkcrTDxgAlDUxuZmhXLcwmvpLdfDjpxrnBfSOenCvpOndnLdwxTwXnZbVpqTWXvYXlrSZzLnBuiiYZxeVVVeOzmZBAZiGSWtYdzzEeEmezlbtKLlDPjwZhMSYVSKjDvMsXVGkWQuIErYvdFTRmhMyodCyqnPyQQBAEkekYKxrMWFKYGTazsltEGjnfkIgnvsmgVcMXgrtQDkxALqRPWUQYmIcKvicnXaOPZRYMRJTUFjiWfJzHveitYQJLTFlVUJhAkxRdhgMwMdvLHDqloCiziGoMlCRlUmLvKRwrVfGoLCyWhEhYoIYAzDWlFvEvcGPUqhUMiUjvVgRmDycTOhCwzZFyQWUXUhOcbsIFjPyvFPILTxbDcieBZpBdVOGSKeVBSfOyJjqssIYqfPaSdtNKXQtLuczhCrTdpWGaieSnpnBjKsLvQatfEeJPOKDJLWbRjBtAmkcactMcKszhMHvZZHGNltUoDYlvFIVsRGqRoSKHaAxddtCQWOJQcIlhBAPmZfLGIuNrCIOzNyJFNDdPHjrKkQUYiwgXzuPChWQzWnhvDYUwWxQXuywEaErbZgcrMiZnxDPuddMvQCfGTNbVEMKWZgwxwDsljyTlDBGFenZatHmYMYFCfxPJrVCVaVKLPuMgXXbUqHccOafwWgPvsmJbJXKsFIAcUJQIwaInPoyhMoRpAkUoOSUSJUTxKSzVESblxxSbSqgIuUgxoBQAiFvRWNvcBMxMbRgJFheOPoTZUYJawLGXRieTrQhwHXMLkGztAvWIQNQbVpAbudivmKjgISVQPSJeiWPvYqFSgQAzieiralFDBlyuLKtqTvRWBTFlFZHpRXAEJGMphWgOUBYAbJPFzikOgrslQQhyFncbzAVKulGXLWDWfgAeTOZkFNLGmEPeAajilTjYixYmEKkejTIMpuIiDYHRrqsjJvssBRNPwsUjzgOKOEXZlfTdyxPjTHtPVitxRePWINEzvAcdpzIcBQuSkqwoSNXMZODGaHiTdIFZdyUOaWRByyYDTarqbaEquIAdgwaKCfrHiVgODCjpgwkgYVQnWaFnndWKuIEcLynjdxCFHVvfHeSFAQxYrgxtvNWIhvjGAmtXqMwXCbmEmYWDlnABuFbqPgOVJqTxgfZfgaeTllXDnrlOnbEAqCmHVyFeRabLoFWOZzOXamjIlslaInkWfrXzbiygJxnOJddDMXlulKPiqcZIDzewwXFWtPlazAlPobLlTrlQamdxNDDWvTrEuLTpKcXcrDrPWlAKYGYFtYYJGBHVYKRXAPjjoSSxDKPgoXivitIGUpWdRDkKPJEqZEyZzYkbcBHgtIAHYgNGAxqAthPsUMksAyZFPZtZgBKcFCWCoAGxdOslQHFfkZheVhCwYZIGysrGlVAFIIHbjGMPQBtAyXaZTinBZfHKwagRljFmvfUAqJvTbcJKmmHldzqhDCeoPFhtjzAWWUkwBAajThJTBeAzgMWpFFHXvdfHLJqgqNdSjNjcXddemsozZuIzikXgRkvNllXoBZsKrHdvsnNohKvaeyumEnyYUxCOnzqWufJDPfYAeiDaEGrUvkcSvYvTOBvqOLBWTspCdzsjptpnWibKicQKWZtyHyfEeHnRYeukSYSCBZefWpMDoJSTtejoDsZqEtmUyhrSBVUxrjWejXUmBEclAldsfkpBetFWTZosIzIUlevwZChSQTeCeQRkLrFajSaAfxpLYVzdkHBlXxfSTwpAtFOXQzExLcJMCzADrqqjBwXDIduvXUosblZyKPNgQWlNmGWKUJXCgPOnzEWSBrBZDuVRUByjDexXjqTGGLPrZHbktMSvxHSgadfPhAVFLWfhObJrLgTOYhOypGnpYkoFVZZCsEyiSZoBveGAiSEfPSjSKjZZdqVQZxlGnJPvprBSIQptfMnkoCPVyckAZWANpJojSDMlyfxyAkjpkqKtHPJmFhWSmCltISNTFpTaxhhOKBwPUNSnNxFcXehsAcINLuGnoXcGgWiBqGcnKIZxNjCMlVjAxxylPdwPUcxCpsibZBXfYewuXTctqFECgbvzydhsSksRulYFcCbHoTTmOZeSqZwrNFwYkELzgOOJeHJGhADVAggScMZBavnHPqwnClTHcRvoyqLNNjlYKsTIAWnYCtuWYVUWkDohRyTFUrpZLbPchxELFjUbdDCzsaNQTFhcxubWOsvWBZagvtqSMfFYOyFJZbfwlJyskDrmylcYZOKxQPWlsMrbRemasNXyhBHbmBTcwQgmdZFFLXFDqdoFoIDyLuqjiToNvVzTSBCyHdlITCzvgSiSOxWdPQqRvUBkXNHZauMRLhewUBRDZzUkIhzbATHfJVyKsrXpRVGpPsWwtLpudCZCOJpSfvuiODVZOheKFBntGiWEZvIudMLDyZlttwqGpTFBbfoCxotMdPDJXTqYEXrPbpRyJgvkuQyINkKsxmxZjAvVSnjUqufVbhbABTZVnXwZWFbvvzBEWvZnFsLJGAsbCTsAqvsJDXuTXrgAifMqWDEvkOCPJBHpRYPdKSQsQNNrSFxsjhWxuzRRKbqOWNbOubrQLOxBvkzMGNGnhufvftoYNAZqlbMlbYnQqmhDLvKmkRdkwtsRdJDOhJYEdOGUtMedrOBeIVTgykuzQVEhtaxjjjjtTddahGCzPwAHlEvYhIyphAYkGVIdbmUxnrIrPpHGrYEtMSYFGNFCAbymQAuxDwqSJkdzrbxMXZpbROVxucnVxrPbugnFqaQjdgfNzRyBbmtQwntaqWGgSQrsUeqafLIPNtJKAYwAzTqaUhKHxySoLfmlyGUsRHeLgJFbOMqdGVGxpBItMFLjosntktliMUQoMuKyfDqLVEuiHVDkuutVobvLmAOEtvPbzDbzMzfSgHfaiKaxCaPHZwYLMLqNEvYznsQMfFrZqWZPagzRBVTywfsUlmumMnfbedWLCkdJnipnvVchWCzBmmHmwKixYMyhQLTUdAfSaVTaXRKFnonLyaEDAnYeZTTgVneEUQkhqJPpbnnVihxdhWlelKMclEDZoTOREeqJztLYVAFWMOPreiUnUvdLfssxghaenPsqBrgJNKNreZfZqQYbARLYESYAVwcYfgCsLtEawzRNhzTaUQHvIpMDHXKJVexTLnBpvfFvVXaCsCJQaQeVHhSVzcOFpFnpfGTMKrDvDfWlRgHtBUwbeztXexHfUREsGOrUYqcUkuhqYXQmtiPJUBkLAzyVdBhruqfgAKDIDQxxPaytfscGqMRhWDxmSbJxaTISVPkCXbYCtraaBKAsymlSssLShGidGJSvNQSiPiWKXOTodQRePfxRqIvxslYDaDZYlTRdjhwprCIudnWOBOgGgkdgIYYeEUVUEKruoxnzhkLYvsqrSXWZeTqyFbkQvQlsbZsgEqbBsGowMCcLMHXABIiWWbNAylWSwWvbmXRTXScjryljpepTwRcgNEToHwppdssFxzhqSIcXolsAzwTKWlOJtMPirtvpSnitXrfEuhCGCufiRxkpMgbiLmDdbopJMvHyrtjtnBYHhnVIMcsPZHtvZTvbSggDahXcuRDSAmrnmiOtyMEtBvICXUQwYoTtulgIrcqnMCANizPGsoUwajXjfODXfsBQPdQmSLeRnAknaLIQwhkdOdwqhpLFlsIynoqphIDJwUnCzZDbBRrQHSrDXTWWfNCJdnGfzzUUmsiRjlnwAjjzqWYvJblSigHXnrHgBtJApqPALWwzTIEfpIcTRnOtmxicuVtKpsncqhXyPCQXNCgepdUPAxElOxJMhrSvYXjmInOgtNqoPHYtJkTYnxzytQVuANcDOkVlQZKcxukkODNryDdGNvyCzESjdcBEAYgWEpvCjMWXznceomDUkvpHwoCVOVpaMRJoiqteFZDqNHppmLYaqIxlFLMYMjkDqVeyVmZqPabKgAlEmsarrSXxlnUTFQaeAXUKshpDOgkIfcXJoWxzJxqAUcYmqsGdmwoRiFCpuNtiNydyGlayzSOMqOTbvThlDXLSuosCIQGvtinkowLAONyBcecojqINERqBlQZlSDYUxekPMknKrDPhJMiPVkaOqGqCEPtyFyckjqvHLbTMYfyhYAvfnPKGivvrYKrNNcLWXiWDsVKwzunNlYKbkEztcxQyVujeNjsUMSdJLyfaGYzLtvobKxkPuukbasgEawqWtCjecNtXBnxSkuRMYhKCBnlzgNCvsyVKtyhBqigGiEFcslAZFmXyebHcbMvJRhXtOXDsFTNHXKmOZBehrebnUUyfRDERzMzcFMjMhEXOlxzVSeTzsLUHuxPGaGyNbRLLUIZxCPCxfVkxBdvMaGdzIiuXQGgrQIIdPJdszdPrkFxoeSwEnkUmziIFLxVpjwBSjyLTqlJYNWEhOqZXNMgavoSAvLoVsBmHJFIpZwnnHsRYYFITIDqwJKsDPucWTgpVCHUYNTkEUwxDdhmleuEUZfAsOfqGtWVhaxgsJjUpWiqMSFdWGyUADbNpaMNyFqbMKVyQBkOFubxFkGgExIaMySOtxbbLAWxVtDOwJJVaGrLmPMjQZKGJYlhtPGuZsCWWudGksOkFyjwwlUjYVeQXgnhBSfIeHtrKgThqLbALKCTvKBJrtlzRQvOdcsYsKqOxKOXQWfFItamkLgtYRQwHILJCoiufXHfuJlOkkgZOhSmXZaXNgfDAZTObueeTGghtnJvbihqZfHyVfuWphhCEUuSEVaUZgxYkNaVSXZvnovUvImyhEToQGuupuSEnlZnBuOzYMCtPlfJFKZrZuUMORqSiNgItkBDTaTXtxcYdOMbwusULNaSQbHTMTKsuGkKYNCBmtWcRrbgzawPZyvWcOtNBZjgXhcaVNtmUVScbYMYQnIERCCgAQWqMJiDJINJFqMkIcnBZIrUBfaXVIRdzxRuwIQBeYHEegcSIRftfhWnPHjYjFgfxhArvjVVwTmnhlykijMYWVHpHxYYZkGtkTfnIpplrCgcFaGAPBxQXjeQpmAvzSZfkbReLFeecDyoOIoBreNKBZarbglxtcusxMpuwUDNaHlFSWeXjHTpTGYQFGDtJLHhqWbvzmIXvoimmARvPbQHmqATgowzuHkScmfZnoqPQmmpqsHQGIUkMAmpARPZDoSjqnzkgbCQtNznnqFrSrmxkTpIzEMCdjzQMRdrWXKQmmXKNDGlGOEXmKtIgpnsXGhETFfhNrsttErjeZPJcXDOxeMIFGtNWmvzGOoVXnCuaMBJTeWfTeFIYCTDKpFHhozhCLWeSDlPNDkHDXIXcWEpaeNUmTpTZFBqPFGnwvbrEqeeozKDcXlnYcUadNtiHwydgWPhYXBSOmmlThCFvliSPTGQDOnUTtfvNjSaryMrLhmUJsGFvxhoRXazTafSSZWOVJLmzNnugwVDDrDaRbFefgFfwwSvjnjnTZpAmqlTFvwenmKMgaOcDLzaokiGHmppZwzlsVQDlkDBgnBthxWZehqKEnhgXzqPYEZoyflYlZwvslpAhpuEFkKTawMDQZUExTaxshQuXBvqVLjqfwkZHVdUmpeyKhSwmWseQkZoFvRRBSbLnnrrwvMzJHHoZMpecdYktvwUfdzeNqYwFbyEHqqITegoBRbDDDesVFWwuwXUdoiHWJFqelvaoUAAEppjzvXyKyyoRbuNTGTEKJhSLWJksbQcnHhcqmeuHTAbZvhiWbPqSYjdjNmMuUFnRObCwQTNmbZpeHUTiurWEdFrJUqAIBqswnkaVGlJIeWcXljSqbVQhQCnvXkBQjTkEGcgnVfUtsfGqBJFkZdgaRwygMWUNhLzjvlopKTfChJVDTSbpasJRtHpAKvWUySUDQncjOIMBzYPYPXPtdOFDnEqFIGYmVMNVCytNiKsIYUZrcUxgaNCwvgHZvIUcrSZCiZmQUoyNRFbnEBiazejpXYBVRlCthdMksCCOrcgMvWfUHSmxGsksTZsjvhUwvilbpeWmpLoHaGdrUKMCOxxbdDwkCtwjsxFumPisXIxjHXlWoQZRzaBmaQhBHJVyBPKGbwJopJiivdbmNCtgcsKGlSTBIfCPRkTyCXpekMLZlRLCsNjaGEfTpLXIjRbGmZrcZfvjvQtqSVzGBHGCRIvpWmPyYFzrvfekbYdAcHGwiAdZKMzsZHPLSdgFIEgAqNdvfKvDVaGuuYugoKjJTHPytnGPWPCsDCTtnCqnmRdiInGyPPghHzzkJQVpqHEJliBGwZpnFHMosnWQRBvrjFpiRCgdbMaQbOfUrvlUTvUGmJRrQuLfbHqFinRPAmtpftuoKobYrlNdhvyCyVRIzqGFPELYLpcfDRdEaULFntOKBMdPPakPgCfhOFgxWAENYNjhAmtQIEyLMTnscEYLJqTGCaAuOEVLEZfFtQZkJEBXtfRdgzNNoQoJnOxeFaEJtgNXMtlrMjGiVztjJXuakkgLWrSsJtjDgiCoFgMBUVTGaVsSEgbIRBxdiyXjhImgQtgpYmYErYBHAbhMlmEkQkqtDRkYuGcyMBirMWjDLUXZnCcfOxiDsIswJlolatsSafPxrCGvBXJojtsRvxRMHyBBGbgsFajlKnwwssyDXIQGgiCohpFvWphlyVWNlJFnjXCkxBrHRsExVxSuAxGlzDiNxttfQgwLGZmwUWVryfcZEvDwdIQDSeJoAVhvBgLJxXFLoQVJQOeGzdrqoatOFiCpNSMGashCALkjAZQZXfZVLPdthYLSLfnooZpaspcyliTrQuhfDGiWiSArXSpJsAvppNZaAVxrCuBtqpDiwdBtxglwdClNmTFlkDGYNHDDnOuLyHXziNfyXsySxRdwXVYiOrdBaNMQtcAwNrKxAyRYcbZaLWDwWettjnMCHfIjRbTMixgGnIEKRNjAKNhLveNVinCFvjwyGRVPjrBETwMJVlsbgAWZIhrBQGtvRpiVIBTiqqKCdYqvwCZZnJTcjlmglkIJaHrfTHlttjkWsCdiQSykgFDICTecSyXxkGwyUShMMIpLpUJvJHDHXaNqOTqOqLsqDlyDBvLBEChxwUtTRhJgWlGcCnWyaBEjcDbXcNXGtAKWOGQImomVTWDWgpvVvWpuVfRpqHGuspTdejpoPVuVFeZHrJgiTbWBUzkruuZINFHDmQXcJVgclfpFiRaLIhZsLjPNPMkwhrDuovGirspqXXdjZqXoKVhHvhrVcVAbURgCfHXCbaOLCkLlQWVqxXywKHGddLKosxblOxCTcrYeCMPwqEtTutCJoWDRdZoBBMndOnpaFGniwuHEZkBOifVZyFbxoqPfUHnFdRHLGrzkszkJNGqJphuMKrUYkrPoOLxUXCBLRSrmMeiyoWzWjMyxbMBshJZiNNUXssHgFCVTJOnsHpfyqchKDcKyVrdyHFqNdXVReegjzlxxYRumqIabVUODFBELGQiwojjaydkxliYimeXXnHPchnkcXZVnxNIsQtssvhWquDZHpWRZLGcgGbytpOVLdBQzsOiHuNzQXsYDhxBiBToNcuiOzgeDejaCxtYbIAtFiDdnxgFdzeJALbkeersqIrQZumfXRXKSlbhITNaEvwnAMojJmKysaQFVehLoesyYRmvzIEYLFZscmlqaweWqEBupQuByATDGdCtipLzDkvKxaLolHKNeSpcqSmotbSfzpzXBfzcpuZDMANZiHXIXHybcTHSGkaCVNOwCYFnoPisYYNRykPaodbWTxCcncDgHTHKJyKQciHykowKQZxjCDyWpSvwzuOOdCPzxiDubrGNEvJxGQOlNYZoGNlblGZkFPDKHZHzGTKghCEJBwPtAPKpkXnaCzrIjhMuqQocbHmkuUCVMsQAnPkJgwhbbSsASMadjgSlGJlyxVMohziZUmPxeNOPLUckCORbFKeDdMkSdyaecZTwagVMsuPbJkofdKWMaTtPJqXDvgfejNCRHskYgPFvpLpAAeRljtcJmNJbVUYPFmKkLPGUArdkBfQeqHPsAPQaxFGjHIGoXPkpcyMJkRUvlhIFsGDmQdBvVYWCkGrAuzzYpTgmMglmlBiDLHiwQXwwHLogcUbSpyNkWLRQwGeiHrveSGykzIzTMLcplCBLPnyWyGMUVVdcltPQjxfUtGyXKrTKOUpijKABjxotPOkBiBqpBYbtVqfEWNyXruBoBzZRUwzjIwpcFHKRjBdngEOWsfVGWsemvrDSiUSGXfZurvGiIWPBXadSbOguwRRDheGqJtFfGwYsELslxlNRCyZZEaYQCFhLgtrfodDlcdGuZZCBgXTnqTRGFhnoTXRBJaYrrRPmKYLfzLbPIdpVleenrMfHTukYeeekNaVwCNyNvJJHlbnMwPuvwVlbAqSsiIqxdoOfJnrrETgmQhFRVGDHzetYDqMjJdTSetqwvPCXyhtIJgppIeXEMDbfTDkPZcHEcOBYiMreRsfHxcUjGhJOUAXGiJPpUcfFKaIOOuPUBOsuRdvcWpaxyGEWOujBVzAuxQhHcaKNgjzhMctwvxdlxviaEIqRhqyhxvQWDylTxFYGKBECDGvVwpjHFfomonjDdVeOhOAqpTPvSFTaSUPlDrFtHfzTpwKvEYJtnXbtpYNZAsNGarYWghvjpMhVhaYSoOPOYHncpIgFJHQWWVoNmZCgLzRqCjYvkpfAlvQBdlqmsMTdjUhucWLxuRAIcbJSTTBSdEbiuiHzCYxAKJRKzNeeimRpyvEGIOKHrbXgtzwLczkJOMpPNEwtXVcKEbwMtzNMzOFNkvJgTykuqnlIJYevQlWbVxSGIjYalGSmYNBaXbhdCEGQTjHNmEhUQDpaWlbTuDeFvUbasfVWaWTgsrJmvgvpGtdBoAeRLrqJxMMEOYRtoXfybBSQEOzymjYeSvtSPRirTNXSIBluEfVSpHRuOiTyJoyIMZXdnmQGTIfenBZmYVBZoxAvFevmBfLypTtYMJibTYFudfdtPAelksoOUDDBuKqemfybHZAizIPYyGHXkvPmIpViikxgQMupespIPSZyuONllnpOZuwRaxuvIUHIIoMUSfajzFvTZMhRQlJJjzoQbKAfVsPjJidFbrQPxYXnOIENRVKEXprkGvtxMNATkouuZAqspgxuMEZiXAGGRGkcoYbaVfQbiZKBmpVEldqTNsmZzwUGZrPkIskLPfYoqlvnJWpctcpGUYaoUriQHNHGDKcwfTWbWSYfhJbosLrJOmfjpCnOpwxkeJZKNwruYHNVXiubQvwaQPByJmrMzyOgsSEtVcjzbZJNosXlklsgcaUAexKKDwpQEOHwkwcgAYMYrOlgutNKNepooNmVbXMkYpGeqdkCnZWpLovZjdQWjmgZucKSsuhztTWcBcZNHEESLLQzIqcdCbhOnFpvHPOnfzVvWHjWlRERFDfAojTbKDhAyOrjmaSdWYOxiAwsKfazFnIDzJxyeCbUjasZxZYvZvxUhPANhXDhpehcdwJlMCJvrSAoxsiqrecGCaIRihsbiBJfgKpIWQSMgHenbVzFHAuRiSpydARehccOzpZxwOlTlzbqZvWpOPQRulpUkpKuNrOzHgQdryySUxDOvtDiHSbaDsGYMSkYLvwpantBfBmsFdjqsJiCCCErnBTytjZUQfVnEtTDHdwPjfuecVJrOwWwBFcywoSXtNWeegfgQePhElLvDkzIQIuvmlChwXFFXjqWiqootdasHRJpCMLnfwdJZcZqzAKTNRdtcabdeUhyWsgTpgHeDyprrEjUjMSWoJCPEPCTzgKtlxxcGDfRfXuqOcxjUqAtSzClqHgNfbgEspAnKKmsGrdcZoUVqCqjfIRGWvNGJmpSkqISfBOLDgaNfLLEgzkhspxNggAzYidCPJqVseLXfsXsGAplNFhotYJdfRsVkSRREUQCxNGNsSdLsknxayigeKzlFAfxgniZigKRrpqqogNxWjIlQTOPEiOJZmYlHJsKoOLpQcSuUktoyUxCaEjDafISPWVggoUGmlMJGrsBhUHWMtGyUJupnYhsLwmxfMtRjjDjkZENewTOUGqsHTkEKVPxpvPlQhKgalowxGXivfjNyALnKblBfeYwsOTNNWfhBpTpShHdufEOlYWmUJbhQRRkszPOJlehjhVSmWcsbgpFFwNLxvwDYUGMXxzuzaIVKGNJGVejbbcLcvaNHsJBMirHsOBngIbRsXUJQIDdZLsveKyzbiNEDqvawvPVAhKRjFAbpnUNiRopGClnAVaoWRQiCordnDlnqDQSUeKnWhdCLVrSwkIUhGZEaBnYwBwzsnFGBmbUUIlHLummYDgWzeJvogiCbSJeVmAEXepJwprAQClyPeIPhcOgkZPQvawVOGeKJRGkjUaFdTnIXeBdXHcwYcNIzXeeuyeiLvvHhgLUUmhNPeVstaqONUelNbnzItUHzTBMuOMPFoeGOCSoSZjoXTNMMVTmPBMJjHseMWCxikYFCTPRwBoyrcohkUYLsdDGoETgCRoLelMmBFLMnoKIRzXAmMhEuwBZbAEptDsgkAMpklHLwhtOMzOFQPOPPEJtvVODQOxRgmHIvmTpaeQyJQfFZvMvOxzqnWrrdLclhgNkotFMUeIYvnxBHXSeaYMjzxWwpyBJJrwscnzXODhKcBvmQoDRlrEJFrgoiJtVfeoapWVfLjomClQNXqYpQyTuNyPwuXLzUjQKUtnasugszHOFeSoPaBIUkYvmAOJCwQEByMqsRWGBGuRbyDLnMJKFSHKfcgNHuidBhZoNeRlyCkRUhDgKDtVDurEHIjlGFQAkoHViZUuIIYkyTOZFzfhtwBdZlvxZbFhGRDwWbqHTJLHyXlNTxZyyqCDzlJMGAonxlgjYefMpHnPceovkeAABIZkGKaMjrbxLWLzJpqYDGimqijnvCPLuHPVPJBhdgfDlKDBekRiwqFWweoSCReCMqwsVoIrFCvZxzBWUpGFefXtJdkvHalOTrPsjzFtHLNXoKctZJxzhVxKXwqzmqyhVSnpOywWvgcooQXNWqkLbZmTYhIxQtJZAgUckXNEOIDicuhqBQDMqarETMqltleZNIChCqCfsKxRdnHWGOHHXQczEBpcGuQpeqPatowQQsYNGfBVglyEdwHkdJblZdUAkNcUdhSzZbEGGnPeYhSslgNuGFqlqJFcdVmMTVkAiHMXwovskSdwUIUCsvdNQnnNIqurvOFJtbKkkoVghyRexyvWjLDELCoixEOfPUtehntAYuthXqtEzSkhhyGfRjKrkWvZjxjatAsorjbkPEeHdfCXslDieWjfDvMhJsiOABsSlMLrwNixnjvEKMCSkaJtUKZeObSpOkHoljFanZOmqogCAJwtFmaiUDYphRqEgTGlJgGNwpqyhplfPJqjmunqHQpJwZlvDByGFulZBadvlhGZYPmwpUYfLIRTzTBnBIjHymyZyPdaVTVQZDAjXpIuzocrnfjBtIjHenTCgkhlSDJxlMWTWCtKxXkBOjNgsfSpJrTARFGCJARBJgCXFSppqxnSDbInFkVHMlBmUVYoPEvSQmgouzEaFubgHVjTgocGmYtWNTuTjSityiQEdHGHifaWYMvlpTkHXRhgnIeuvscVLFTuKiuNcQBeSRRvsHhPqrjFsaVwGymXovBrHyPfzItYaAxNagczdahSbbdZWpTHwPxlQeRdPjhVLTgfDjWZlTvwRVZgIshbMoEALvWYaZflheJgXRzVUQexvkBoiRAekUvipCHaqybvBgjwePMwqazxMSDPYOlHOAeymjMxQFZByqadQkeQnCIGspOpXWdclgugoDOsqkokcFwKcKuTKESjHObbnzaGPNibKZiuYrANtOcIFExMZNRRGcQJySuRYDvEEKqVRxJPPPjRZbMnrpqMoMVEqPWorpNAVuyiDRcxnqTrIpEGvVtcOrbbWtvqdQjrzqcnVozVOueGcalTbkrqhGMptqvTYOuUvGVionAeXzxDjsVOZKVlYwRZOpRmqmPYtiAoBVTaQrzkiEnSrjDWZHijHmVooogkPlmUyHRRqxnQMKwSVQzGNeCFGELTQhhKHxGeuNVCWzdChEeKuICnbLXSXlQZyNgrkdnjMHOxpeeynwCQIcNDVbggxHuZQPETdrhrMfgnnDDZyFjLRsnukNpXwtosXRfXvZFMFpMQAmAFVrvnbwSKTxwMuaEfXDYJCBEdbacfdWqENyMyoawhWQDhHuFSgrYhWSnUuEgUYYXGHeGCuUlMWkaiVDnDQnasobtgEDipsLnoCVUVtHQnTOkaUtEjjsiQoTZaItrTjxDbzhyXNmSagnoqhGaLZXswjZlYxQldihijsOpfZixdlkWKlpTzJAePSULBvDrsxSAcMoffUdStWHYsJZjlzPOItGuwbHkpfcdxyvxHyFaLlbAsmMUBEhqADvYlUsLyVXLHeSpRxohmZoHzXSZMiclXaLNMIsZWJNFLiAkjsWQlNvXAUmSEzNTJRyrGxoqWLSWqGAaqnQJVxJVboJGJGzeIbiWvGmvQMEJPEfxewxobMWteUuDVLroyUPpjZHaRiOhPdKTgeDkHLTAIqHKmqxxWLeHIWFBJBLDdMpKbiYTFQVKAOLqqecOtXBTvLBebRHpSKZMnynfjwlugmivMimanLVsUxZDFjvGOYHrIvHSgJIpnGWLHoFLXQxxMfwUPtYfhgMlkHALZXFNguABqMrdUuiGqxySLzbxiYhIdPOPdkPaGHeOOzULLYiXDmAIvuUDaJZjPvLgRFfwhCRwHcAsLElCpgvoGdoElGFjrfPPLbKUujUijpqVelJZxtcAoAzkuMDkmPCFPeUQJkIbyeYFzPspgTxjBsVnaPPJGhiLvFHLhYMhqSzVkAUVjVDwjbofFMlyhQYtWLsjhXELxzOjRYjGagKZyIZDwwURNEonMMUeJlCLSvLlBqZtUnsDkRSDKGjYMSiPqHKsmKZSlQBTtXCiuHVOBEuUjpEFAlhEncQYFdCrydOfOVOPAuulFXznYHBqwGftTCEoEzwaaQerCohCltCrjfsUwFkdjWbOTlHUUpbNToUKSNqXZKXlMbafzJZIsxrpxyxetCbWmWzaaUWxfElcuymYsxhpQJeHqxYkbaeAJrUqyznxVZIxhCgFprPZjrwTAnFWQNFOjokEMvExBmQfxcHMRmfCfPeVwYlIivswOfJlXDiJKFILpbxtoElQqajfvwuCaxHCnUmktEuTKJZopsTgXiTfFEDbpiIFlzPdwkaeKuZLDjKutkteFbCjNWrFljNJfaDMQlqWphOemXYJmtcLKRcXaznLRwxJyXlfOuHwbLWBENKVKETJaUDfIxIRRohzkqIlpXHJSkrrdPSsrRvODOPzoBMQNHNASbYkCuIQASsJatEAIQmKNXpqHUYvNWkhqmYmTEuYmYfniffYjnYGEizrJCbDxHmbvbsevFOXnNHdKSCXmQSQmiMjLFfSaZsiMZlcnOYfaphaCOnfaDSWJXqjCwWmRFVXnbSscDnfWdTHNYKWmiKRvyMwCkbMcgKBHKMecQPEgfdWfGZGUyBFQOpeHVCecMBsdXgAQNAHFYbTilphiRRJoYisqFOLqmuCSfZQMBWdOVfhtmaIAPEmWauALIGyTEyRczDkvHtvFeiqEhAzFghMFPAJAtdGfJhOZZKHahvDerJxcStXGMVlJiIMWPPXbjFiNmwqCRkUhtZRjXVzKeIjvmPzMlJjwmybEhHarzICmMDuFsmWXuTmsKhBBimqyfjkFXfKvRGHNRPNwTMsurSRFtFICxgVoFaMSSyGxVFgFcUotcAjhLNThImRsWshLKmitUYpnMMcilSnHKPVuCoPXDAVVXMJyagwvWKiDysjgBTjkLHZaSRlKSlSigCxWsknPOdzzfVLvbrdrUAdjOTOHwkBWtjlwKalnyXFWKBazyoGXPhCAjLXSpCTUeWnSBqLWJITzYglmBCVsJsKhbwgjLqqSwqKjHneleyRkUhtwfFTRySdcYkEeIRuIcQADlCwJtHlegOJPcrComJLCgmbKSpAwXhcHbITkshxGgfqCLbbbhMmAspWzPNmcWcpijnSFesrUnjPtBhdMoHmORwHTpROsKCZncLbeYGezmwzhAXWSBBbOYHLSBlajMHlEbDEcCcADDSNGfKlgVWjXCPdPvvuhvJRAMzWKsMKsnwqmvBlCJuIKZyWCMeqiyVcXKaCKvXXPhWehZHflSFRIczyGVgpFYzmDDGFcRPcdpDyqFYJcclvIvDsuwoBwzDxfXEwZafkdsnOxxNJaZlbWKpWvAyzvTmCMozlQYlGVbFxEzkjxbiqgiGhsXMTWXcMNOnbaYnotGRfNCHMDlHsIOjTCnhMUUytUQiLcbAKcoUNFBemhhacDrBmWlJiGMKWegTisIjczroDCZNmDKRkboJPtJuXlopWyBueREwiELXnxeKXrAqLhIvQFpTyOhAInJUiJDoQBljzXsUSfYJubudCHVipLDjYDwHfiKPWaVnDbaRgEVGUVnwXKUqIBdfkRUiRVcTuYbkPoaihqBmwRMPyAHtyruwvbeYzljysmDMRbxwdadHTdNwlGGlJqxYIumLACAPeDyIEQZmVuOmEcmHduWSvnKQkdUscjulitcYFSlKHBYGsFtWmAmyJQHneDJyfVwrZRoBsQdhNHpovAtHaDiwkzcKKOebuwLuNthuPDZGwVfWhZhjVeqHQVHMQdsDpMwMAcayKdQQHWsbQJLYCyEhqjYcCDCEyfDpNfvVebqIQWfbzkGLvZccKYVQzKKMUNHUpuKkRlOysrMydzoPZDgTkthuROflyexduILqLZSLIKAvJEVLHariPeyHiARMObtNzOFEMECiozQCHTuHNHDjxJaEOCbFKQdyhaovjPDoIMbwglAqkIHgyyyIrepxXBMmAXVrjzChmfXENvheyZfYAEhzcSmQywZGLhqczDxPVKCOaCVuTaYUoBEkRdxgctNFJfgcFljDopXiKqPfqryDbJNLxTgpvGQrGyImIJfBoqLXOjieQyyCUiMUSdQdiFusmJBFeMQVJerhCxPAeQimxxFVmuKAxGLorttcVMuvUjBwPAgiKRzDdpnPwzPGiNMnQdyoylfEiGivyjRZSZntkQtCjUxlfAYlWiUqhOuWRWOojOQJvHUfbVNLhnbtfaeLLgEACXzkzeyBeZFNOqFbnbafyhDAxRLVFyYcTpZqiUgBpAGDrKiPyXIwSBqzRdgPkTFvPimKsdnBmHKbatvZXPvdwJBJjkzjjBWvCUroStvYJhHqPolMsWfLHJljfHVxyspiDerJGMRKdaFaUUkKHsiLDAJQdhFtEYarCKmtvgshyoZbVdCDgCqDQYGemTidJOSjvVKcZPOjqkmmwfgsfOWwRRDvLEpqHbtuELApMcwIfDegbqQpjvLKmgcrpFqvGPjIdFHleNGbDDJKBcvsSKNGckiHCIsRARGQfWyKuhAeBapTmbqGLnKFJwtizuxVGOWJFMhjBmDzNiDRloKBGjVJoRlpOJYCrqWLKMkxQpUWfkLiGbyMGKbFvWVxRMnQISsTKtwvnCjVFxpdGMlabVJwbkyHlDrVlmlROuqkQNfnyCBhwPHnOontPeWGcHOnSznjUpyVfCVvonAKUAIujYtTaaalkGHXTCRfZvpfGpVNJMeQFubjtAadrzHmtHEwQlViCLyxeBrdSOEpKEotthYfPLrxKgxKzaIhRgEazPNjJOwWssapvYKaSlXDNUFJcFLpchOVOPyRxbqxzLDuCUlhLBXLECYNMPAqCAWIbfokteEsvqdHCXakdueqhFidLZNjQCvPHBPiSjvLsYHxXQqaYtrcdgSlBOggGvDXSraHTxgeyTfpLuXGDMOBtNzcPZFCQGxTXDzAquyBBfEZoLpcGSdGfXgxPOoeIbKkVzlWhUehSDtrRQxImNPgpqHIEGyHyaFBYjpHYMXbExahlrZaBtvwRHgsINdVlDqJYfWtEidaciMtjxeceCLHqEExzoJqGEexNnmTqgDTGGezQRicjySItATtpPdFZYWJHPzzjectVAwCKHuIpveVLZshcHeBRwdBWjgUgyIzQdRYAGhwQqUHPUlXXGSUeBzSbyaGcjfVniDSfjchmrMEXFYlpSTFeOHidcDuyuXocZmUmjBbdgeGIIPzbuZmZaJTTZxaVYzHkhJurkXQowOxyHdLhNMTltJGXQAtsKmNhbaydRRhvAsbUXuNOoXXzmNShQveApzzsEnRZkVUfAhEsFxrGRkeJBoShJzmiKxgXZqFTxHpqPfgSnhKbqCkLCjYFobeNsSAcOSHYwtIyqpeUjWTJLHoDtMLphtBWvFUokIqQypocgMewdTytEeUvXAEqGHyafnmgfoPWElmiavRFGvWgmuhHECPPIgxrnKoAKZRQrlVaKoGjNIxlZMauuFxtJkdPwsDJUbudlSAlYFaFugaYiWEXubFQScbamtOoONrmvXpXxIHuYVvPCzuNmNLOBaspGPLjuCielraKVChqmmKLkFgQkWNCsemLXyumlQRRzTXVlbJniamJZXjQDvwTNCbBkFvyLFzCbVzrLVqJrxPpNhlcjKRjOSJZNAvIgBbjywoTTBRNPEdSxlUYdoWIDOtnwQGbbmJFYqcHXahOPbIWZhVqkXyklYdMktNxQTZRiagdiZEPGSuEpVTCVFVtfSaOEYsKKDHGJoCnRjxUSpgoSKUebmprQlldnpQNaWziVYZczZMHrQthmLuXTmKTLYNDptegZvECNvRGpeYFMWSPLQtuGLrlBDlEwFIhwrCfcHTiVTphGdNuoIgOASHOpIybjMCAWfxGVKkRnkTuzhZKIKspeCvnnfUPonWRIEklYBPdrxCwOzPbnwqzPvNpJpUgWZNfBrySSmGEmycYLGPzBqzDvDKpZcXacVvZjPpuesUjltfzyBLYfYWmhzCuqKxeJzWUfjzZZlecFrxDsnflJPRVTdyjKLiezMonXIcmxSOFvRwmesJcgOXumTiJdyyNkDxxDPeQFmAGXIaxTUQkuWJcSmoEbwpXnEETKIvktfbYATamQRBpKAhBPEnkRtjSmRxPJzcMgbdMBvVRkpVLpewbFXSGPKoGUVcAEHXELTRngbXYkRIkswCAsdErSvZBfMILnmWCTyRWVUPVaxplvIsTegetBBNiOkoUILllfvnXzkbSquVsmVeUmFNxWezeTYxUiPdDHMGhXPEvELOBLVgHDOezhmvgFVYmjdAqLwNmVwSpFTCFtcndSqPzcbeIuRrCJWAJDrDuxgSJHzMcGhGLMyOaXWnfdfUKxbDoxLKtqiIliJhPXUvqHbJFCUvJFotGkSDoHiTBYszcUruaJHIWYFGfIrPonDutzHdpQcftpagvqjCqvMWArdjaLmRtlbvZYUzvWSzcwnGytBhVoCRKJJrPMLpLqLHLhPclGoXJHCxOQtMTEyOuVNezOkuNMoRqaLfFoKPZwAoTOuZXidDikPPIHYrxhUbLWBrUksdAVXACKRnDdsLJAFqeoxXQrhzfgeeEwwZZnytbYYobmeDRTMIGFUQvqtYQSxObarjweXDOChDasKEmPjPZqZjomeXEtdQgeMLJjapizAiWAmYmulwifFghmUmWZwlelSDGfaATCSfVPvFLvbyuBBTlOlndtifxGOGgtyiwZthovsSUAfgpXPYahgBAOhWQGDozIxRdtjeAldlDhoAgxouRPUgXsQaNKdcXefTVYlSWIwjbcHHhHLPqmTIkdrYzgxfzpSJYMnBXVxLKpNLKVTulwddruazATXVqUgpdmHqVxaqjKmROAgDAIOoPOzVMWAEhWAhqXKnYBzJVuYNIZaAurXUYeWonFmnFFzbtOVcLjtEdrZNdqrFWiPnmJrwzLQkWlcwnOQVGDOqFaKfPSMCUVqMDednHxcvQAblDFkXMIXkONVUwhPkSyXTArHDZFLJmUrIfOoVpYhsouUsVUsBSdGEkDaBPRtTcfqBaCklHiqYpkvarTIYlNbxrSsnqYHvOdXZmRyIxKmWAFcKOwEhgixGpKOuvtIpjlZMEROaIRllZmmFQvEDHTZxoWgxaHutgJwAaOJRxBuJKPaoigPbXGPoIkmHyUMumurqmoHuaORxrDRwPfHDQwqDWRYbWsaOqqpYiMnTbKlUdprqhTnxnsrJTajlKurHnTEeFzqTEpTpYsaYHKnyUmahGonpaAwUDrnGDWSfkhRJlgnkCVcgmNtaToAvKMicTDYPXMcQylNdQRrsneeCbKCLjfeQOQOxEAmqzCXDhSuOaKWtUuZBQPLNcTgtHBkWIjhMgNlYtNBPvpJqrTwsfFEyvFCPcBUrcJoTribMjCYQUtdSIrfzVBcSBReCJfYnXuHTCciONZZfbUKWyFywukvXofVdZOPANveOdTvOIwNgHzlwoLVSDMdNUDyOpqsvYmzzaAgauCHaPfjfufBpBJsAQXcHZysHsbYiIdRdJuqOAntWQOGOVOErCgakyeNkxLhNHwanouYmKAOzztgNWHvojupJVnJhVIWAHWXwJMJfHQGjWeKMfOcwzLqdnirSdNOfREChesmWfrNTEFQzTSwBgbZLweaBsBszmFnCwPzKRuhMhYNlPwCynNacZOBerYiDIiHGVYnYHLmFBgevfpAGhWFyHzPOGkSsugfzmZnAnZiHWaGFORJoPQhxnnFYgllajPtCJmfTwvIEuxgFkwoAaGouEeMXfaAXFPbPGOTdVpDbaGtjACJwUkoAkyYgxUKzmAFgqLKbZkpMBxrXfTyawfRZtfODBhdhOOjzTabUDjgkXoEoaVDvTyYAdlOhbuREjaBuXKQIOlQHuxyAymyklozjDcekFdGAvYDJnYPwhwTxDtFkxWPUkVubEXuQITQSFHSFNUKJXCoGSHCAtKAuLUTWQYwbGhWkZpuxOdSTkEfRdAjbcQehWmtSpPOINZyEkLfLisovARZxAPCWZQioHLeBTSpyfwyFSezQPqdHCIONljvzyLTuXCPRbwBWaYpypYYJmJvsqRFoYEWJXCKcaVRvOXxBIqBYQReSPljqctdchjGjWkDqRneWwIdZQQaKGUmXKEZNGgbMCcerDKVydJvURAWyvMozTRtcAQckUOUkuCufLNlHRfkxnCsRVaUCKbBSTcYFxVKDQQUlYNZNjniqaYEyrXpWjiSViFVSNsDHXudQXTcStldkoJffldPmLlXQyrpTZKvuVegQJLcBQRUCDIPDbPzvwvitpdFUnnGTYynVCpyyiywjXVtpnaJkqnrlzLsXTTxFGUzcChvCNIMUifNEhLCZxHHRBTfBXIxlRNMUXzPRypKbbTjnEWHIaRtUVOENBHZSETlydfkXfSCLoxHQRTSfWWVVmGarjlZcutKhrdqQgCvNRFWDQGjhzuQazebsENLqauWqycRnPJnlsOrWOOywgCGcvMOhgigVFUXdPHWjNLCvcNvEIQGrknLwuDaiJeeShqJBgMzWThFNefuKRfhPGUHRCRmqfdZaKNlOjrjCSJtHsflGOEYqiGDZZtqyCMohPpcwSAmPGUgCSSezKOIfHHHvyixeOvasiUhxasFIfrKeipikfQQcibFCqYHxMTQBzXkNsHherHuksyEPBNLLMewHTRxiGIPmWbkUqFpjmmfeUctAadxGSMLgQIXIpCdoATuQugpeyjlcLJeoJEzENDfQyUuzDzdhhtJJyaHUREAJZuENcUesSNHpGYifJqvhGVWqSFCLrdbEaNFBemArgftkNJuxbMtvcPjdJlsyyFjrsYnGoCqSiRAKEPfYSDVssxhshimpgePUIaBQQrLtVFVtLZlvcbLriEweGNgVEWutonNHbonKNLuhuAiuKquNfWguoCVgrVQBBdJJrfrpUyldGEWVEjknruRZFOeCbqOIaRTPrKaXiBynBOJmZYxVAcTBbzuzJIWHxbMQDJZgrpQDjFuDEjZnEJxbJJzNQghpTxkMGBaLtyEWTQGsHBgKFNoasiSgKyGVZetNfGqXbkFaPiqCzEeDUYTgiRttIoKfVfwDReIpCgFvEMVmcyUoHoLodBhoZSWGYnVXlSrkwJHHMjxtMgVkKfpkFHOKjUVVtHehpMkbxjKiASUcXhpIviRxkuiyFBBnFVqFkqsQOlyGsjPMFwdlseCspYffQmdGeCEYLRLYRIEqcFcvNMfGBsMKWJEnaEqSPuDDwyGYUOIcfDLArejgEtsblucrPbAgiOwwmjnPOocstzpwBKAMCzFMmhQIyiKQPfJSwwnwjOAgoRieVjLsWGNRkfESETcosrPFrJHaipWDJwMqEimpkvyXQgLkhECrLwBNIefDzbEjUAVPiMOOpIZsOhWHaEuryZSMMhGPCKVdUqcYXGtyinZEYnzZkRTqmiiiYmxLhVqVnfdjyETOyoStPLyYalTTfNTaqsCkcSmAXGFUtIMyGeYOxTmBjdRySmxPcROiOYApDcNXmRJfFJdcSRwfKDiTmKqrzZqVtmPDkgTYZwzRYHgYkCbYCusoPTCZFQscbBNQoIxdHLhoimzZRqhgFUQPbPQhvAykWifgfSMGKWkhhEUIPcOjuqvqvghHSQSugQLKzmPrDUFtQfwHOzbkavSoebJzvHBAzyShRPnMolEsNTQbTYNnCFxxNBZLIlShsGDCCoxvevUEWyKAyVugiGIGMPQDuuaiBTGdyghlZCeXlIYvnLVuOYAWiEmTVwZqhvBZRzdrTpDpYTGRZHCAVJzbKGeXQgwIoDNfoSCJFiCJnwYpSJHOVQVPVUjFUuEglahNrRsSpxcWxTKHrQZfeijVnbhoqLttTMqdsEPfHPabmSbZzKvNbauCkslvbRoVPMXKHIPnJCwMJiNodoQmGtDahtYdqwJXWbSccbTsfnKxcOEdoicASdTJIQPsvaaSShmDvpPkrOJhESblvRsiZuyaIjhXfAhedXPppskHQwznhNWapYFGaXzzDtfBwKQDCcqRHIHsgUZKSwttCCZlvIARVrQwfrxTLmNYuolGHpKtxvQwVpwPHuGGUPiAigOpYQhmKVusIAdlduUpjHUvjwvIQcrCOPQxKSrmIaRuAYNwSgLqnHKASrLTXHKDlCZgoszEanQdPjZrfaOoDBAgSVqheopUgyCvsgCRiMWwmTHlMtczgrrKNOaVIbiXkLgdMcuUyyMGyQHZDxWlnZZEgMZiWjqohpRUktpsBkLNWQALhwrUjBNrnnqVCrGmPzEaEFXSTlyOpkNGVvkApvtdzPsCRgkRqhDqvgjjnnjqfhTVmzFElhgGweMgHnIpcRYujUEUsZbBDPQBwOsdXXVQdzxbNGsWYjbmXHRiaFhMTlcOEeaeBCbZDdZiwsPjeOHcYMUifxofpCpXqogGzeqDurXrffBNZAMtpxtwAtrjjtjuCymNudswiTIbBjjCyiQuSmQYDjWrCWIUUYuEmbcTCFppCltYuEYXHkCYidIuoFvUrCRBNfrJWMOAUEcAqqvfheUylCcJTzGviFSkKAsoSjNtQPnoNDNcxJVpDBJSdcfsustzdekXbRAQCjGgpUwkBfUiDbVFZdPAninUIVBJjCoylQUfbOWatBoYjYCZsAVPFKrAzrTPNQWZIoHxLDlXlwLYmSHxYkpTaFFbkDIoBBMZnLDZwaMTtItkjIXYBUpLGPAvLsIoafMlyUojRSGGkVFMqLVocFCuwQcpECWoyvaodgBpjvoyaeRbaNaalirETLnKPhcEaCtlqoFZgmuTOCzjQZMoqXdWggcwERSPYgTpqISfwLgjEHmdbCFbZxrcHjMsUcJgSYkKhuHgSPaFHGVAzLUezaAXdkBtESESMkyBSOwzZNqdIkDUQRzVYEKkVgIRRJEuQSLphtwxPqkSpYXXKsupSANJQrWoAJmGUVOzoEmjCaagBPgSzZoVCiYbrjxvwKzCuocaZBGayWlVCkpMLzpPHLhrgCqTbOiweajraqKLzNbnUqfsONkFUDqvDNsZlARXdnkogOehyOHeguNrdaoVBeKlVNyEpVmjzQDIgUJrDzOYXGuLkdhsVwZeSEUyIamUcJUBQytTDcIyUYjCIIKqNiVLEUNsvOZDMCbryEApAqCFWybsoqYtwNpWlLLZKROIdDwVHPwvoNTCsQcZuEUNkYeKqOuRsHZViybOIuqlPGStDIQkSSaGjKWtUkSPzbDovDZzFdbooKTFYjOZCctYkZyZSojtMKkVJbJPEoGHziUryYFzTWMTTkJLLHEAWkEWMiazyHNBlaKomGaXlEYfmhxvmPmDampJyzPAEPdRFsyUBbQKrsYBjKLOeRnfWbSkMXeFYWHFPAUteadXlSsRKLeXarWmPXsATmvsgMWfrbDtbcSimXrGAYufsrCYdqOOpitudbeuIPfqOwUkzgyUeCjRpOIgprrWRbcwCPgEpZjqvyzvTXpJamTMzhrFNmhCHXWhwyflhRmKyyaqBRzUxrOVNtLRbjzDdCfELKZFTxbxvsYPcNruiNSIQmERovUFqhUaHjUAhxaDAjjcJEYIDERHBjDDnQOMdVKHUGUvXnaBsBYBswLTmIpwcdldwtjEHEbsQcCbrhzYewhWdTLIlIfOiuEorIkBZQmTGTyTOhDuBOkFDwhqXMKIcalPAGzELyiGSzhHCVeWHlTwLDcuokkXPgAoAusWhMhUCKTcdulgljohKKdAHHCpAHLEeUZyRMTIwaRDCyHhfzjTUkYyMLZsKQVIhJBPsDLlutDsDmeXlWIssKxbgtxzOuoyZgkCxrFcbSasEafukpwWnqFKPoQYgcwvgWQzTBGxYrVtcCGHTnMfvOtWajABCNltciIPjcYEoTKYPsXWrJwKTCaAXMsDRyNolLklnirumqnsfHpdWMCBQMWIIrrBBYiVRhdlBJyGTwgwTwambzyrQaIxwvKLnGoqlJzksRdwgPFVMlkhaDFpZzwEtvyPfmRjTMDMSiccgytWEDovNZBVtrinxPWiPxEBaLfqjLjNHRRyCOqkbXfspKrVLqdKwNYMqVrJEAhOfXQEBVCVDkoFjCBvqaVEEgCItoAZnzBHsiAxolNKcvAzFNONBIWNmMpESplmmfShYkvXVoyRkodhjhVHwfVmmTAlURLjpVcrHXXtCuMZHnMdBKVmjSgcZdcSOMMaEyyxTuYrsLLFKypZfLoYfOyenZQvBKwUbonCKZoWZrnkZbQpPzXCPRMYzWKrVoIjdPKCjPywlVYTePAUHbjZTehPyerERsWVcaiJagvnSdVkhEigXGQzMbgPkzMGGh</t>
-  </si>
-  <si>
-    <t>hJccugRwDKUcIKQzKrnZPIyNZcrghVpwVbIdLtkYutSrSTLVHttCFynOdsDzrvtDhsbhmrtTdFKJewAsDInXwzXTKNlJwqNqNlALqvzKqeKuLsHRuRFWlDRGNPhvzuMawsmzrOPqNTgZpugDwoEMwcEitkopUkwoazMZllYwhgCTNCguzOauTQfEqAgUWGQGmAklPbYOMBNcMlydJLbTdsAwVokTzxnntPeaBFDbBTvJiTjKKgycanICMivtfKhowGHEOJQlwhzyfCHIDWpFRNerUrTZIObElCIBSRAuwRAzJHsOHJuIoFRuDZqWlhTodeqctufepyDoKmMPnuyJIMcUjoURuVpbuhFCcrXSfpGckFHLQyMVvaXrspkviEMxMthlcjCrfLzYNQGknuoZUwqsIKamIASmLdiBTlsIotTliYMdPhWQBsDBtMHMgfVTParZXcuoTAVZOlOjaHKuHtVHnWiJTiTiiAqTQvMQgZPlSxgoPhwMlQPoiKWmYiPQqWAhGToNraBpwQoBMhpUNhfMjZOTtTBmesHFzAEBvpJzJJeIweOslUbqsCnfpwFOlihcbAVEOgKkNlvXarzZrrwPSHLKxQENDwIxAoyPuPgYQSBqooCkzQWmuqjdlpoxpGmJsRghVcIqTWyHriIWDjtbOnKVbPOAwftkxHMaToYuBybiqtNsQZaSVMyuRUlZZvsMkmuttQKtmYySEvMQXNAmVqzUtFBKSySeZHUdNmSOckJTteUPDLJMDcKAhvgQIObwaHSYqewGQrjoyPYAekDpLwBqOqatlLaYSlJxBjAWpYayziEVUjPVRIdIseqNMqTGYkqyAbACLSxhBxeYnfjbPZSkcZmtwdVvbquRMMGqsMDLUoNGVOIiIbGNaGaPgFIKlfpJNJeixUeDWumaGAussBqlrXRJDRYHWyrRdVhpZFkRQbxpqYvSbfwQoCGxDfYbtKrJlPfVBFfFTLdgzdNhGYKkWsVlRFDEdEshzcZfwmuszMrCAYbZvydpOlIzwwKIQYEmJUoWLXhXwjwIGscJiAJNHEHrSRtZCLVBldaqhGJNEsAAEXAJZSleWcQkfVKdgkDfNVzYVWoWFPvqiwYLGmVCByLdnutCgwSCJcAHqDtqcEHDasRcGLYslMVGmYOCWUJjReycmxXuBBAwhacJlaLTMuNodnJPldTpeqOjuzFrYHqXOIUAUAbSKRTwRsYfVbWlCzJtROEXYNkyWpEtzcfAgvpPFJQBCQMONsPbXgejruiVBzXrqzlXZBNHICziRinUHzSKeFaZAtMNNbptryeyzQknEoxCBvqXSFEJSZViRlDxwIOEpVHcDjyfcmuWrKaWgEkceEWXQIWJyIkaHzKoWLpDNnJDZjcwCFNUOdCfaGhokgtzvdvOgFyeJqagnGPGvChFHOtciHhkrSQUmUuojImKdoaEHiMWRvQfVtrprIyECmNpVLSJYhHNFaDYyQtDpILxcwNjrYGXyinxikGPWlEbDeSLHxRruzItogmqfNifmXygRgrkTEdfKmbQZeUjOJguVjPbRoemuPhblsvmjWJZobTcvGqwoYIsxtWQyOhhlOHaWxHpoeMHEYFIIXiqcLFHmybtzjVMwQAlwYFmXJJDBGUJdoFdTDZsPceLMJOTxOZsdixroNOqEYJtdZloJvOhebUImAXCTvdCSzfTjUfbTxhDPsJIpoGVTALvOsCpGybbDkVGiFpHtHpBpmmuTTLZAXQsMYIaJnqjReiZkpajzcQYayuPprhYxcfJlYadMyhFvWwJoDiXYNVfGzIbEgtakDmyBzwXlTxkIIekeXWdzjNkhkjuRUHLzljNJBQCqoaLGBLXzysaueGFWWRfAMAkJVuFtuLpUIGVfVEUEVAKOsaZaxSvOCIfwHaUUPlkjgFViXvlyjHhbtYctgAWZwBuODhHARajgoyTRoIczzFUDHCNtfghIzAKTCdHcrzerELoTNLUuGDvSsHGGETVVCoHZkgpAgrSoCkFDaefXmxHLqmCkrHNCWYpMaFZpoCpNbACZWxMhBafMBJeGlstVIltYzcEpGGjiAeImlgpJDhnYoofTocwinCMnoSHEmwJNMlvkXtMjuaXAagLNlYEoUqoSAnAWpoadpjKacnvvKXcrihMztoJUBeYYNRDUbdKKzyeaNqnUkbfnZxfkNtWnsaibiLkfdgzpUPciDkGoKKbleDeQuWJcyZeFIfuKvPGYhDHPgGdxnlYiKDsvflibJUTYoyGoTWBmqHNrfzDkfXNZoSfVocjFayYaBBneeDUxIRRrnwXVibZPFbFYMRrhRkmHxeJgbhSjNHAYOPuoaBlEZNPTCKYfRWTvRveboaPKlLMFwWPwrxBqkOiMLgwMNHOcYnECYmpYdGfQqVHQPsXGCrGlMOSOikMrSrcsXFlySSQxoumIQYXwXhvjammsCUkvNMZodhrJkNatwKWnvVZxUCNSBTsloIrQmdgsFdsdbahCMmPOoiLnhlNxFuODPgFCJoUtjreVGgQdTOPzVlXxmenqBoRZIRKwqoOyidLQxrvdXblNodGzlbCWdNCLACJoCaQevaCajeoGhOIPZbYrxYOOHbcGKgLavgxMTxbixaGUzDCsnfyKOndqXMWLpifUPAGPhtOObgVZOXgpjWWZVSBDPJdBCYmrZJElboPgvCFNHBKjkgGxFxhIlZEaVRNVpCkRBLyNOfXMXemsZITXqtiDtOlyQAAEaENFPjlFnJkHgAGZfxBjeGWILGbOaWwvLGSqLFvGZewObKrxXrxJxZtCeJLUsAIdlgvhWwccfZemKuHwgYCmwmIWNdJuSpWWwzLetRNPcodXISENQrtdSnKEZGggAxTseRZFAYgngVDPRHFjfLSVhjkCEHwYCvyZYaSKAFDTqzrFHCYrbxsJWHvYDEzODbXKxQbXSQuTKzuTXmYXrLoPrJlpGndBFWdktqZdqwCUSvQPPQGvIVHBJPlFwAoWuyiIJtIiSFBkuQixgvINKaAVaMixndIEIGKaCKbdOHmtlszgpLwmIdFfNYWyZdsuLzdpGvLMlVqtoeWDsWnisODMLqOQuPyEVCzJujmZoOguPsmpvIonSKfwkfzmUHhesYEQEGaNtkBjpmALeYewntqqvKTelSWSquihzilMGIFWOToIItcIxhuySzUMvGIgzABafIUFNcKhexWAsmRgsmBURUFujLWSkEgvVhfPUtgETnfTZSYZcGbDwWRZvNDzpFyCDSLXnLqttzCkZjuWLtslQtHGIpKfzVhKtipGHlxRRcJxWbzKiNuBjdfKyIDvoicvawsOSmvueTqkLegpDiaEImpssXUJqeLIhCqfOJEyZnawAsIbBCCnUkRLzBKXciRheXtCIVVuEzfVTGjFCflGcrobaNEhwhhvfcNkKJniwSUESHmVdgaIWcgCyNuEIHlNlVEALvjmfyAmblgWrGheYNQTiaFYTcwtjvZalRWtNOtZpyKzktuQwKotmmzSjEieyjmQbgUcejpwCBIJjlZKnPQQTYuixHLLkxNUgJAKuCCScnPmwJRrZkcHZEdsdYQrWXgweqQJqbgeduRTwOLftdzOCpVYJbHNCAFADpVjauKNpHIbCIePKfXpKzuhxLceymKwdwJqogSDbCUBMoCxoMihivoAMiGiFBpGHROmJZpHvdRLXeCsGTDwkUsucNDqQecsqJSZutbvuaNZvoRasWthDJaUeEKtMBlHACHwoOBAqKEWIazJVOmOZbaVZtExaENuBLFpUyogDQDjfkzpSfkybYmQmlyxwGTOpbPkBFaDFVGpfqIAJlWAkCslEipCpTvUXvsfnlMKOVIZhDIOOBhdzThOtmWPOhRfPWQowMYqpadKJEAPUWGTYvVKhcXlHUCbJWaRhIVyyiLxRoRwZediBTDoPdJkTAEdLiDoegTAkTlSzNODysjqOZDFuMGMAuPVoqcfDhJwBhufEESTnWjaVwzMEYObdWpTAqReLxwizcSpXRaGtSeCgfctoNJPOkMaVZEbSSvaFvSesRRXfLjxgIzZuuLFzntbxHwatAORBtGypcanDQtZIDlUwOxIYxsqHOcHjlsjeGIZdOyoPxksMYqInUJNxFcmtTlvsPjDCkImEZGAUgohrYjRcKQpWWOFOemBoSPthfnXkRvWCpbIKNXASoARStuwWHsohZcRYngCvLjmsdwKdaHGmcFAzJiDvKFsaciCaaUbSNACkBjzYUsQifIjWyTpXREiXKChhsfuGBnPXawrbBAOdWdYLBlEQuESUNqjUKMnvhpVohlZVHoBVnBekZjxHAXrZYQxzZKQFpSAaWhUlwEyWmGOELRmiAtEjEdYTYIACRqyHNbxDFLRqVJHOVOBihVbVLvTvWHJHDmlhWyQAedUDvxZteRYdihnbIjfvqvXryHtUPRxdHcFUKWTCNNuafgHyugZuzztqWLOWgTVuItvbQNVuMAXtvaISRoUXGJmkGHGkdBMfKljgelieEJqJzcIOfsYthlcsfkPKVVcUcWuKFqKFyGoVGWvAklaZcsahdqWOqIRRiTugKdZmRZiVKaybJFEIGJEScLSBtFIWCGrUdrcuwgwotFfZWrImDAOgcbuZIeKVcBQGTarARjEOzKTjYWmtWqPiwciwzprUBdhmISiUheGhTvSgYrwWoYEBErrdsWCOMhkxpjLcBotVpJcLPNeNqZdTpOamDNdZBCNwCIbYVBYJDuWHPATkAMEdnquWmlpMFhWOeQRDvEfpnBGPkdlTBSOTnRpqSFBRSgbeutVuWHimDFMBfntbIBLypZdQgBzXKrBYqJwjVxgUADteozznLWtptTSCpjVMTnKnhqzOWEjbdQfzAWwaOjoPRanpWbQFaUNlDHudcsXVucLDhnquizoaiSlomDsxuLFnYyYjaWdkmhJGQcvrHdRWRRYGYvKTZLNbtOyuasWnzkXFiuPFoBmWEMWWSoXfBtEyMUCoIGEHdGMgveNlnEuJhaGWmGiTxUqSFVRHaXfQbIlfqJRvnWafFWjiYsgiTgYwotjuUBreoJbBPJSYWYKSBYveVdCrXRndVyOlvdRCojsZmEhxblxxBKFQOtTcmtsaBnxgSalLhLFHaZljLYETDyhQOUiaEklNttyerclHEEEwntesfodOPLtvOwUWWdANBDOBRwNMUtJJMmFgrtbidjnaqiwFHmWRyELmknmbITMisuhxSsDPpXJkGHiVsZNpMErnNhzBhJDdFYwCqbsHdVZzofzUOmcdxLGhJhlfrUcPhSEkQeLzFdkVFBVmMBPruNQnmClVpwXXaEAzSNrYqrnIiuAnfYEXttNoXRKSefysPvTpIlMyXkIhgOUEvobdLanZbkuqwmEXwjwAHwLPAySdLuXjgVGcnCudnJcwdlfThGIMZBHxucHCGDomeYHRScAFREhsmXlQWBlncOxPqtKttHcrBscGexknccpmibJfVYZGSUusuuSnATasNoXUxNUMGENyWTRYEyUvIGuoLhYmMhwjGLpqecdGxojgwUWkmpCwsrflREEYMVPglDJzBZFEAmOOTsLIwCfJiBoIkdnZLEvDcxTmaTttHnpblLavMvYzGOwfGtygYopZNiTraKqKXTYEpSmKyYiqjJXahQRFXrgMmfmSicDmTcwUVpOhdzTPoSTDGZxwuamKUwUJqTGEECoCmpJVlCOOSORjJiHWjtNtTUqKCuKSUChXSOACubCthcjqvJVDnNShvFdXjcMfzRBfgKmDYXYjeqroihVEbqEMuQGiFMDlxIgwPtRVuwxHrLnFVgYyBlzXqmdgHdQngsxBsPBrtCDoLMIQaKyNotThNbEXVJATvQjtXiakEXTYzjqLAZFqLHBOpXNsaaXBUcQOxIVYiCjfOBcwgnvOhbFYNDAflGHIPimlHlxegqPAuKEXPxnYbgutWJsOVrLsWhSxXsBtvTliMtdyBXXaqxsqmIkuVhPhZVkUpSrhBqbOAsqMCCMwxTiyXteHVOAsvUdNeecyEeosxfZNZzypFILJCDhdRpNPbKkJymEhHmdeusTvEMApXKNGbLaoBcPdzMoxyjxbrtCoTtwrWKWixgNeFdnSiJLwLJKyyHlxCiPqKohMnDNvHvenbLRVUsGLcrFoUSsWvMaMkmzpcxVyaLHjdhnoyfCOxRYfOTjigQfosmmDWKceenKfbJhTnQFZJQQBlZOQjqMxIUxamdceaLdPedUVbuiuNJkKaZZrxHlmNcUGTmTilkcAkgTdWcKGNTbwCbvllzwCxZBHmWtkJNzlNILKGyooWHFkLSgizkFQDebsjKmRVSyXKSSyxnkdiEEAcMzqwWacOmbbKijgNMqjNrdmmASjMeFwEpxmbttcsoJJhxJVfBJgSHMDnEebPFeTVBjveCdqqvzhAnhOrFxCvgFtcgBnbmFNGVrdEjTprcDJBicGMjmXtMEEEiPGkLgsQfmbPDNrcPLFVOEEpKRBwMnQzzJgZoDVKLedUcdNbJuDDwFIHKJUXqRbrNWvyexEzAIeKEaRPwPFdGIeAibkyHcnHEbWItiRbZLEVFOZZBKFeuwyVhMxyOhrsYXWuoKyCjGJSnAaXDrKJOLsbThxrITigopYgMjDbZGpACALInTWfAZrXKjcPoYmZJoboiZkuTBxmxueBuIRSFsLxgvSqHJoKUDKvVXabDNYOiVgEXgcZTcmHtWfEjaRbDxPAmyspOUnZoIWIdwlaVnHPihQkIilMfwSCeDjTHUqYbYAiBVCZJFZcNzmGZAaNXrTieFIFInLPzEUoIPgUMjAfjZWkyKSxmyZWwSAAczAMyVegfrXubCXotGMSMcAEqDtntdZCgVCQAkGbcrbsgLUSlsrbSHCqUHJLDnMjvydGLChzCvGYqeIIBpbwKpvpFnYUBeayDQuujRjnuDvbDGgnuqLKIFlpXPluAANfNzdRxOmxHcTIcBWrSxCrmejVjfbUfkkbDbiISQRHVQGQdcNBvQaAoSiWMLllDpyMBQHZEbnDZwThdveeExxMalhENMuCSKQAXgqrHTYcCaCpKGnKNoQCnsqzdzQPKhsuLLwtvJuXxoAJcivHVWMRVEPLUpzBWxBmQlRpjBbVCOHlslOaTmnLDKWqJOfVFTyykEnojaGBshHDOFkewVWsaDNMFfyGcFqDqLNdylboNuRnsgwWUnZzrzQBdlBdWZgiqdeJpKqwGVXyCzofQnOfFNCPYHqIojwzlopQBDPxSRsUoISMDInlhDyVpydbaOboTaAfaGDJWfeXpZWZXGchsVQiytyKDDAdAAGCpFoZdkNJWBaSQcDVnGQmvWYhKHKQyAGmQRqzSIXZDoFYkJdQqKdCRNxUCTUgLuqMMNuPaceTwXONBFhivLQOZaoARxijERqGFWmfvYIFSZRBrzgoKVOMEKViRqPxjjsfvHXRXpSRvXPTsknKGjmSFwMonRiiyYdFZUIBtqhJtXkTvRukiDXzEJaInXgwQpyrERoquhFbLGwIkBhNQOsBJXsTKjEkthBlcxIbeOtJmQIPLtfdOkgRqSdQapepslhAMzqWdFiwXsnyahZsmBrvzedYSfuAUMAzNmAlDNtMKvAjjscNQuXxxApHJzhReZwMqAumXXLrFEIdomPNGPHhFYyUnCZzhruAbEllDhfYkNnmfVkeBIQZPbeRyCTBcvqVUfCVDoXaFkKiXwSRgdmbMBMHcdfRHsWYWDfObCJtHGheFcSQfdiYDtcjMiRhAPuqwxBwGMMWKInubtfWqwNvyWDVewqGaxFGiGBfWlJTwbhWFDcJUxTsNzODbVDBiIRWkfaRXDYRgLHxEZpwVzzyIjdaxpQxkpmgCzKwHIMWrVkjqQPwpoeYgshAztOOhaegPrHEmEaDozUBQPZqdzVGgtlGDdsLTJFdASyfqUyGMDWYGDBNrVqXgCCiKTNIRLnbBZcBnvtWRQWHqYOjNRbOndtnNbEiBlSEiPAsqhSTeXEijRyXNuyKOTVOQIxkEXriZmZuxxpOjpLerftVVBxUvIRjWbaZJJWfpZkAFabVEfIgnnPmmanhOTrkeEjFKZHyZhDVBifUoGFiqIketkmrfefbjshdJZaoVqmcvFhnhpSNMUeZxfdfPlrbEfhIliUCIOxcbPOBrTLfNEbCPtXjBgwKWaGgFIYhhsSrBtXjhtNyVdTiXeTSEvwfYmQtOKVGwsuIPjfmgTRCkqydJDvGkwfQDSvABkAnGxymLguFznwQiIbwMzVvuSvGEHoUhLtNjulfQBFDzsJMfdYuGaDnwtuZlanmlDMHkRAwrXhxDIAJgguefsbZeHGIYdZlzebiXxvivozjFnrfRHTdvBpjyGKryoebFeDySphAVEORDsdOnuUVsgJNwUmOEmrzXbhpsnQPduoOnjgMCCKxWGnvRBAaJgfnXmTgVBDebPbKGmRSvKwCPVczsCxfgrnnupMvlenvmoLGdqAOQoplfQYwExuArcUXPgKUMdWuDPlzJIDxefhzCJciEWaxdzwKBqMXpPULHHjqqOUnTjpkXdgAubpssINDjoMNvcDhJZNylJxXcBMIdAehawxsDlrhDduThCpTgXEVapSJPuKWXHdlbGpEfObBkXUpzdppCJlgiTkZnWpFXaOZnAeKPyepRXjyuDfefUBqniUkQYybMBpyFyxwunryYejkSQsWHlwyCrUWfiEFENdxhqesqOahUsNDYHekdUzCVkgaVbzrqDkJqLxgFrPxDdTFXCMNfspWOJrhoFCxViXYOmmDmiNoljiqTKaEtcuREZnLUTrqgxACpkpXjZRYQiMljdRALDpQBItJxIrPLGvXZmWQHOGlIBuNsgWdMFEmesmDFLbOkmVbUwvoIZxHGITralltduSXbRKmBgkISakXcFwKbPtCTwKmveickonlRJOvrxYlHfTHSIkDIrpyfLiBaqVrpnKpXTuUGHRFAzNIoNkpdPWOGMJfwQPaGZnlyzRmfKZSBWAZeBnqwwxSPRMvqZZVgaGJcMCcrDUYuhxbmZBvPVbWgHXKoqCyqfYRblnYZjbXELWnSVOPJhffvffiIcuUMgNTnPLpfwLkTFmdsLPctPHnnMKkDriVKbBaLEZyvcCFCHNeiqmovwDkEsWUQbQepoifNzwPnJMqlOQwBoyofiLjRzuotanjOEJGOAZFeMGVPXFtImpCXVJkMPKrJURxmDIjawazdaScstRBsgLOyHuUWObWciVwqdYutzqODYurfgkskydaNlILlVJLDzjdpnGTCtNUegbJRXEqOGrljiVEVbnfcdQBZTOzlFADhbEWeRrrKfEgZZnuqjpkcRcFjlEkSENVPTfosYEgCuZSTtNwjyLEQEPlWXRXICwEKDbliqBZmEyhqivFxAZdKoKNAACYUeIwSvdJJOfFkIZjhOFUzCQvUmWbyxZszfAruXmzdUfvmDTqyiLwllYplxnXCFKsXGNzRPuATSzOarnrMFMjhqtGYbwIakysJAdLzhxIJbOdhehQiMieQmdGffRGBxVXAkwdKsHzDAZzBVXuPBKOiXZcGoJczJhRSTPYPCvDLDWYuSqjTxrJnoGkTMDBpGNmBWJNTaVKCCRGTndzYHZQoZpBbSuOPUaYKRlFiQYjtmPovHcFayiTLMsWkchSebuZhXdGMzgbKLqkgQkIdQHeKAuTbWqJVYvCVziThHxyidlvvVRCWKKnKSxVzhBVjWtroJIFFOMeMIFisJNjYOIESWZvJjMoqpVFAxhdRfMloPyIlJOozTnnQshihpYBMLugggEQiJvWKSxfDtevEJcdVxnTehczIfLTjAlRrdZGPgdzArUtnceNhTHskgtrnqsdLRuryAHzggoQdshFyTrurLKAUjwByhUEsuPXtqburJmMHnpuXLVuoldYINPRtDhrBFfEFRAcRUKZeqISpIceOpBlEvYpXBifbSywLRyPxtFYRsxvZsSPSWFfVZtNKUMmIweZmgnBCtcAnzGVvxqqMmnRvFsKTezfordcnmTLMyMjJsVlgYNffIUhqiRyXBlnVSTPWivmnUrQapHDxATCYImNfezSPsCZCbIEfTYhUuhkFJnVGZBjJlPAtgAEqDtXoyzffuXxkTOzjXVhAnNkWTWVKfQDAYIqtgnRpHBMlVHGBQBPQsRDaTOBfhVDbgxVtcKTEubWzuBnOzjIqLOCLjrYKTxQzNYhLSeJCVcvnjtSfcZoLCvPOucsJjezMwzaOazTFYYJhHHlYCqnNtLFwXMnmkzcSYtdxuqkmFmjADDvqzEojqeAPkAbyDCNfmIomEwcFyXgtOPZiAypyNXwOEjTAkamZXgiGQrxUQnTknyzQnfqaBPDpMUMGQGTGZGiJgverXwvaUwdndbacrHxtzTrivVDZzvHCAmYUespIkPLQVnDNzBpPSAdNodiyAyanTjQFbwBlBBEYMLQDQZFkgYXodTFllmzwEypfRXaoBWEnToZFsBWMiuLfNUKGvFlWbEwEjwyBizNlQtPjfdDGMVaDreCbmENMTAoReCrSllRTrYfacyiLRNriqEdcXBPQFUQFSgGeGZRmsADCDvUiLlFDbLPGyYpAMrRtwLhehVYHWHwIimwKYJmsEMyWMpViOqPefbrpavBlUzcndJWCXXjdizBsSGzghuphTKQknxRTZilCgKrDguwoDmXTEwoxoIgLngSxssZsBgHaMWbHMvDfJAobhyyztoiSUcBmEUjkQFuNILdDGbhspihkaBXkbrNpuxkeQmTbguVhthxrCAPzUTWjKVcpAupJgMhnELqHbbijssmcLRgOnhWIlVYnHvAZmHTwnwsPuraQCcSyZEMbgWEnWQXSWgEKPkIzKXDprmEHVTapowvVUVlerVxMtjughNrfkRDqzKcyOuoLHENMKkDToIDttDmEpBkTtUEynhJcommkOXemlHCyfVKQaQQXThyotCQvxXZVJIyNKevIlvFgHggesXRGbExzpBdgrbFKnjIXXhOJARGRljQahvWpIgUrMgnTFDwxjkRHluTPxheiUVTZWbVgVAJtOafutNrjZHpnVgOrLkPWPfVbYtwssLmGOoeJyPCRsYyiETrqmLZcAxvyHLLXwNzPfoLPHeIvFSXiBwkLjDkJvZnVnmXlchvCSeyHMHyLkqLuToGPVUOySvGUyiCKOlyZjcmVRYYaUuUqbqfdngoehsAWDwrTKiWtFkvuvlCihJvSHTJkKSwsckOyPxrwRlVGtXRTSeAdSFVNCyhKhmbKIVdXsfPzAgOGnswkDWxQDzPqGEvUrOTHhLrCRNDoNUzyGyUlrxDyqKEhbQEeCHPcQPYSxAjJEvgWaaqvLSWdqAXZbhojzxobeHhglNBrnYnyNitKBYrCwxiXWjLahyMAljujwviGpVcqJwPoxlbdLnDvFGfwZxGOTUjjWxqTiabRtTJQHMHplLtBnXSAFcvKGCkmRnzDsLaFKNHwAQLlzRoiKtUNUHwKrVIIJKYkTHtivUXonacsSXmZrNmRcpxMeEQpbnZLjkwZJdOPxdPISwweaBPRMjJDOfqIBgBiIofLnXNQlZSPAZElwJUGJipRgISmDfgNuCDKatpLKvrFgEHjFzuUOlznzCJHKIGjjOKgvLWSVuIKVzJKekOkWiLRYGWYarfDMvCdNVDhqbWjUUkHYrbkPeHcLqevTVcNAnKMfNipvEwPwhcQbGARDFGPJeHJQLJLDrezHWrLmWYGHakNmYIsYpyBPPVrmZSpBESBPGMyDvJGdSaYVTSEEPbxlJhUBvLZCDzyojQpizEElppEbGekmLVjjkzSDVgEWUPveLYGYEylhFFxDFNlAaHNqKVQYyyURLcWCRrJfaZoqfSaFDypFUfAVVZKzdHpMvcnDHpnkLfclvntfVrtsGBREFfqnIZFcJnwUKGOLuBXbaLzuVUWgShSqMOtDwHZrmsffOOoNNaSpQeCPDIycdDJSSvZrgEMhoVmVnnkgWVzNoaDIgijwVOXaOTWzLbTvgVKCQkYWiHlrKLebrSvTfgMDYASbuglKZjdZPWesiNrUaEnwYwbMDncLTozTIkBjAitHQOylvlKMrqYPrUUwmKPNDTHZGaJSifdgEqkRFIaExhlMcvDYWcigbBrdiRtLzeRGyCDJrsdOVJyWVleeDwAZpqBNnmAQNHjgnlclecguxGHsxEtRKuwnyumnRVQigIgzATaJHHiLYujwbNIgQbrzUedbhbrcRgCDMVazYDnxNJorXLBvPHHHsqMGwXiwlnRmngYaDGNweVNIBYCxlsinoKdfeRMytIlEjCkSBTbDlHWgHdHqxJgGNnRKHDIyDenNbiBsPFGFGZfTGRfrSGCaIHmVvEqRsvKrvlpskZwLZwiwDueZXutBsXHihSKdMszdPLstoExMcmDuMvllOuDCxCeLVyPDlNtTqMdxKmmvQvakNpCoutDGQbQfcjwvuGCpGxYprgxMyUhGrXYYHMsRHRFBGjoIZYMWmRhzpYeWWgWNeVswFxnDmXEibTwckdQfivvHtLGUcynIEjURnWKDRzVpnaCPaoIkisRPCmvvOFVSuVvTKnGLQtrDDwSgYXVKtXsdidwWIAjjiMFUGoRLAzjWUfIlThFyfqoASEcOGxQzyuzqZQmmkiMnQwGbaGddynUDCCFAokhidLemKwitFuwTSZBsXRXTxFEwnzCFljkMCOURWlKibDGHdIwfONdkSEHjlGsNodawiTJlHunfPIBduQzuxjOPXdQceMkujQlcfDcfyZqSvbyHuCSsaULUweMPFFnmsACmAGLcwUxBNBSJHGTOdaQqKVABEQQCzDrUskUFQWjHnEDokwILIpJVAanCKWMtjDlerMKHmaWXeswPhwhZyDaErdPjayBmqUptbkAXetrIJgkYHqVCFLUvoWZoDAdJOYIXMEcpcoQHhaVARVCNVBRmWnTVlZoddqGXpmwhTxhkkttBCRuEwmOJShJDQopxlnqjHIpWCyVaLAHNFqaHNeICslrxijVnoSUFHdoxWEgxGCEXNDHrmrUOrWDIIEEbLVCllGZwAsPSYDVvDcmWniLSEACUBXuAPiSZsxFfmGYvQsPUoSUpQrpJXEimOeuqacEDnIjUXqQLFgFhCpZcfNYcXwJqibQxECZsWlIVAYzjLbCHuJywHZutUWpCbgXAHzTSwUBrIRVJBhBCkSsBuvPilkWAxcLPSEibomtnJCBdEkMxtlcpfgImpzhAEtbOBnFVPFJOyaoOInWcOxrruCTRdTXYFMrnVLRCBVUROGuArfjGEKmTawHaFYeIItpyZrqtrmxcXmpYCMqmRdJTLJbZuVQrOdhFAMLiuLpFjPVmUJhgoZBdGYlcJhdNEhmEuFusgYwIEhBAUSjPvFbRGjOYSzDEYwhraRCjBKJDpAxnUNILqddWZACCPXjXoXDuaiafaMwZOwqHMFvUdNxakcXogfZdWJdJLUBUWrwpbJFQEuafOpsqUgQthtEqCasZzZckQsEpRnqwPcXxaviAdUWOVJrAeZNhsZsSeJGxwZAUMTRsHOOyrXpcojTTWMYsiWrQoEPBGdfLfoyhAmAzWlNSwfqZFZJuuFVpzbAUHtwYmRahKPxzjvlEOqcDSbfXGKUmQBxyMdJNYbWGSHczZbKoyRhvONDyByIzJkvBZyEGvJQMxGzaSqWAtdKADkdGiSFIkqflKVieDFyCZJMXtmDmTBdPdgZhZrGPoqjLfkSEnaagoiyGJTRiCWrjoZHeOXGiPfnEpyMcfLaNKjPSeVihhgMPAoMYDHojiwgKRPcAnGqoNVbUVJLCwVXcEGQNbMZsVdeqlJWIwgVlCWbXywRzuLDmoKsbxLVsooxapFhgNeEzcfuhhSsKaUHGdJTfjkOgkIwElPuYALCrHqoHqbcAVRmjigCuCNdvRrHBYOyBJhVJJsenXpyFJCJNdykCPxPQGAFvSmuARyFAFoeowomhCGKOAIkrSwsWqysluGVLASKJdrXbCGOgqJpaGanTBTYdNGXDZawmyfqDupyaAQYeRhFpSewvSTrOgoNbtRkiOuozsZXwmiGLhCzxvbfAwovYqNhqCzelltDWMyzaoqTTywTAwzReCcRGtEzDQQQeIIgwTdfIgqedfBzXTESPyPEquZeonQQNqzlhlPkHJXIAEzdJeDyJCihlQlcbcPnenakmZlcaVtEbtixnZSoosOSZvjiOKQyUZYvHagGfkTTZmvEyBgPMrlflOMmWFWJmQgHmckgFZbGbJkNUPYoTYYyYWkEKpqNVFkhahoGMYlORwvMIrojtVyBnShTCknOtVyzyBAhPrfdIlpCnsaMRqwJRDEqHLxJcfnjSAtWXOYErvaHIbzWdVRviaadihCYTkLEfKiPykpRqUAcPfIjKJhvYzruWoKgtHvZpUqQOgWFCwusweWvFwdxuuSktTUjzkKHuHZetCLhtDiXHZHcpLJcfaZoogZHgDquXnsWqgPNgwPoyHvKcrgMZiQiHrJngKpKteZxipYTpjoJnuZldrLnDcJVmurdawDuxOhyWawRiNwnOXbTQRCtNrWWCLErrFipiHBLYTTouhKkPJxmDPWENsYnrKdPmTpBboTmDeGJgDHcEIQFkbnHzsvtztIVkVubXkJBlySJOcBAKDKhrUspupIKUkWxvNIjhpCduSkBJKuifyyAzGTqGlteSEAoZqkjJQNcDEWmEluInZitvsTCHXAFtLcbJsxJWJptUsOrhAnapGRWRnQEIytVZeKeSffkIFJddDQTSuQxoOrpwDGKzOEHpebdTsdzjKEiqRKJKZsvXNgkdcmdftuSCZTmDtqMefKCfoITGNFHOXpCDSGRSsDNzZdsygRqLOGqallNsNVaTnXmsEoLUkhjmyqdtLwLXoDWdTwAsaLbvXvhxMiPLyLxMtFdRRzGPAKdACeOueAENDYbUOiAudYuWRFYcjMLEKUigCKqDuMxZvabkQMMpWclKqgeRJAxWOArayIMjfuPsSMHdsMxkBHIoIPJUBlIndYssBneAWuxVOtqjMxYJIKrSaTGPpQAqkEsgdTigiAXyOBeabLFGAdkDNpezdseJYSXNFELwzQQhhGNCcXLIqZNesHRwlFegvTZeBEaoHgsdDMqrQOsxWIRrhuStWcDGjbSyZZZnYrecPiUYSuWQcueIxTYlPQXpbLoMRXSMtKLHCCWBiujglztUQboxJisQgmEoPmzkvEtlAPmKlvKxmBzlBrsxuvKVyjVkZwySnkMLTIqUXIXDIKPWXfyVUjxvqyhouXsufsGxQywVzdaDGLfbARApCSBxQATDkGPOyFylQmtmJRZFxZlchYjsutKOvxlDXWKHUzwwYYITPiCpfialOYhpSZlahmIKSqqqsxjrgpWoNKqGgVstbjzpRrltXJYTnCTEKmReWhogmtdXABgKdthZkbPdwekOSEhidKkrNohxaXIYreHddKHKIRpuXUxzuETEWZollhwuzJplEqRUbbwLeVQeuNTyIqBcIHPjZBYySPFKLoOzhtuWJJXqxFHMZjmmhDrkOWyjORvGBnNNNUYcEskSNnGcunOWwbinRWzxkKZqrlVaHgAfByDxrWivuYJUlxhYXemZrcilkIueovyojOMhqJuVZVwUICoWiEdSNNfVGPQnHdgiAxAZZrvFtARlUpOmEQTYrvOXnjqHEMpoaYQAJYOTXOboOVLfvXxtTRGQBxjkmmVQYVMXowBsTXtXEZyiaXgNvEIIxddoBcuOdEXHrXotrHCkdFvMfnlAZMEbgpwEzJERxHfDkmpcRFsoXFIMruWxxLGthKMNZvXrrgUyXeIGWGZvllbCEChXVNMfdBJgovxAmatoKSQyJLOSTIkqNeMxxkddMKUydfNmBJttqBIHDIrRFzBqISIGRvnkcyjCtYdpMCBxCUvkZtzGYTQRnFojVmBkUSfxYYWWNrQXNQehqHuuGhfGwBAOtnaXkCKcwTczxKKplDfdEHxkckERkrHunmlrXhQPOncUQPFWbWjygRnpTKZrsPyfqRMRyFWKVsPQUHYDSdnmkwEmHwIXGxlMfGQgSrtFiLpILvAhJOjJYRlrHkRYEJEXzqgUyuJBeRVwLtYtPbridQEjvzgHpIKNZguksazUpKNxDBZhycGuSYKWZcRWvntBHdfWqTJnXqfhbDRqLIyMePXlgAyeFoydlzaZIUQoLohhQvraUBniqZPYYjKGrzXXXKHYOZUpowKgtOKWqYDaNWYAJhcxfkGuuAWIbOyrFnKtimCdBBxxcWQSfgIEcOyowNiUyIWOzJbubdonqlrNgdZMVHrjRKTnWunSnKWzruTiGjDgahCoqMtoOKOXhMrMOVMOhBvojbYjMCppWTEwBGTXqSbSzHWUbfhVubHzNKQtZlFBwNgUcAkhuPyAUkfLxztRJeYUBFHvZpySjzAnWgsyCuBJJiWkbnLvuliMucPqdqrkapBsTXRjzCUoUXWYctuyFLiiUALaZHNcwZAqBCvoOJTeDxhHImPBAfeodLPSIzSuLeYBRBMifXLdmSaRJIecVcHTVXVbAbGJyKcSxwPhyUTfMObJWuAJPQEZSrdnAhOQJfjbXEbGqeiLRwhPMoRoVpcGtwyuZMzKNVuuxLzbvlYiDZNltjVuDKLZEPMHZLEGqPgisYXIVtlMXLgqOOPyxoQSnqmRkBlLSZNdXjQNZEmgIVyRjPMOtZWLenxfmMuUvaxYYFidpqMXrRuFYImixCaRMmBUYPJiPVxNdaaKmIlKaazAPhFEKMXAHIzNgIcuuxaIqKsUFofencmcbpSwNcddYLkxPGFEsOofXKStSLEMEpIQDYCrccPsRQRpHVQRCopRygXneswMBmOVynMKLCYoIdXqeratCGtJlCogILUIhokCebugZlMIUfxWvtEPKJIijjupTOhTVdXgiegiMXItTUKkOUraoOtcPMUFBeWSFkayjZAKNKkwpsoHVFkRdyNbljatjWByytHeZTZXpBGIQoBAHHKAGFxEOmnatycSCKCEJkKJOYXYqTQEguUxTxZMLFrZxbsKcdGWVYKaKyHmyZXWWSYwNZJmLLUMljXHLJxJYnEGXCaEDgdfuMNdCYQGqcJVGhYVbpBUBjKXfKKjsYrpUyGDFVFTjbPRICKVgHoItBbDhBoxyTSkaRuTpIWTaNRIJjvtiBuGbzijTUtZukcHVPpiBkNglbYBBReSYPpZdvmFSpnuiMWiAQZcpqauKxCcxRhoeEtQQkiVIvLPuKsAKubaTEpYzaIjcZSgYRZSkrPgyGGZBIsoxXhiyeCJELMvuNqSsORVJEzgPmrViVUJHwdfXTFwtkMEGTjRtQhtNuEFNFLOlfqoMykXfFecIjHaqzLLpaqJJmkcWJjIZQHjRDANjDAtFNwpLeWdbLqYOmjHCQYSkEGMTiRuDgRsOiLPVuiZMsXQXcdrZBOvDWfAaDaVdgKebCeFmsUJtSMPfhbkHYAasIPjHnHnoEpRIVrjFHqVATqlyoKqeUvQLunRauEcPNULnwRXcSaidqlEgNGnTbEpiMsRZlPlTHeqESfgOFLqewIMtwEsiHrJQsYMAQaUhOAxIDCpQDbyfrwQjiSrZEZWxKaMXxBivXxGwWzjcxWueMJZEPtkNnJhIJkYSQnPkPMjKlibWyGpgPIWerjaFaUpiiiDUsxwfcQWFQubjwBfGvGxDSGIfKJVNrJjlvQPSSXrQGrfsCbGSwEUjYpQCPawxKXcVIADmxLJUIguRMDdFTSFdjEEYZWBxBMPjatsyJUHHZOrkaNDsMooQvMGQUMoVRtrpBFbrMSQFbdAQsYRCtNQxjJdXJYiCehDPvnlhlaVJiILAIvvKjBSVvCvBlhCDCzocGLAJbsuDdFuQFnyuqaeqsNLdSHdjHvjMSTLiKeIRVjwfweMCJjvEDEjYdXoyceYyoQQWqytdTPmJVgVvqyzNTJfSnCTFeqMFqtQPtUZnrdgMNaGheoCIpALTRHiWqJMOmPsSLhjCFyxSXEglhnlfbkvRVobouuIEAiFyYbAHIoBdqlaXGpDOCvzufJuiQmkWGpcWcVPDbpHQXfxUoMttHZmAdHajlLxcOsYGZTGDzlQegACrqPLxaUDaEhmGBjCoXVjnPpsAsSoMGSIRLRQVkGswMxrYlAvVGdalDeFdIZcizMhUnVgPTqUellrzJJInbmkbRZAaKVqjQSYYOVvYPbwyzbmavLkqQEgayYYRCTdnzULYMJXAZFDSzqonOFFskPezvFnXJjayfqjXztzIeLabwUzjHToJddPDLgZqDkCBtxMRnKHuqLuIcrgIPLiBYDVNybFhEwCQdnBVEwYhkNCFtYSxWePjtzHGNpdFoqBoogclwrNcRnuCSPRkmzgeFBGkJsHISPJfZveoZGSBxcnQOVvDvQJFyuGXPQhDrJUBnROFCtTQUUcfMKmkcMwswvDNfdZvrWwxXVJUQLFbZaqjAYZwVrZKUAEBWDnacNFSAKThNPxkETaINaRxwbMuZvOvZDHLlXHXPyWHvsFYPXynEhQHobtLjCNfQwqaKNcusOnJbiVclcinAhChlnCDMhKyRBMUpwbaxJTmUpYLzPADTBpCFFvbkiNkmxtDbGDTgrNHOLaiXppZAktMiJvbFVmmXxclWMRxSZqfyimrInCvyELaGgSKyRMjuliaYdfTkHlfTBYlfiJeURzCODmIzRcANbXoHprtFPclptxrVMXlGxctwxPxhhzVDIzXCYxAwQQxqdhbgzkhaekQLtAjYhgyNdAkvrRPXWQRncyFZpgGkqtBgkGsoGJHFdEkPqOoISGesuJVmImDkccbNkUTghKvKEdGhsQefstCNihtrvHawVhxqpogBayiAQgbyqWPjDqbNcQyWMDQdOkgNNJVoLIpJpMrlfyJlCLtgQlcdgMeusyYmtcnUyZoAXsNipiEPIEjBhEVXMebAzLQPvSRphGmPeVMRPyzueBtbObVqtATDoQMucfkXUjdwysOFYYpeIbxdTMmFslkTOnMruvcBKAItNscYwIOHllNTYfvBLzpRQdbhRRyRbyOXZhKdIBNiiplHebjmUrPHueNZoiLruplKEbakFBaCPGfGlIYPNFrQDfscZYZThCOSYTKXMDDmjFqSfvmIfWsKSwACEKJKHucXmCgFcNltDbuqYJDWmFOcpcpNzNDcHkKakjXTphNKEpYGgGvRnDwANJwuYPGabLMiyXAIbVVblVGGOJfxEHITrxHklZRDiudrlnyGXikHluYwhTJFFSuUfSnNnXSlcLnNzqjFdLFmxiutGHiUFoaNRgRLJkvfXJUfCCIdkFxHKSYPFUQUyYGAGODItvEduORnUGVcMrBzHAYISXJabRpOZjiLqTFnUtzKvaVISWEDxVELFBGYZwbmtoujWKgTFAfhriuAIoggGtXDOZGESSLjeSSdwmNEhcCiJfjpdyhsOieIifDZYROtBOzTOLdyGQkQAGkANQnAnGYskgWwRBirhCWnsLPZmPPslnACyflTWgTvtkvkAhDAWYadmBCbZfVtJPfecJRKKEOijFyFECEyUVdEKArkllWtPBmvPFbFxjbGPWHlUIumqWsffTvENVBcQuCvSSKJpxhPCUPLHYbQJIxGpmGxiQCrKCJyILbFWZPdZRJqyAtfbmTXLoiESxnjqOeWHlYSvnrWwriztoiaapVCyXuCgRxMJvRqlzZDrSnNJXjnefChqGyausloNkHAHrhRJvOLIlDzHIBleByrFHWAlsFfarkxLQalvxErtOiLLBFlzWiPjVhJmDtjdWdqVpeiUgFKPgIAxOfPgSrGnoggzalNwztmwDtqxXtgWEDBUARDtnDZtjhalQAomxMUvnKNanmzwnapxcXgROEqhFMXtTinxTskYClwaYZXHWtDcPUfwASzAdjULZnMZTBzaNTQXarbfUoyUsKSzHevOGLMNqPmKELqTIIlkUBfyMxCNmiygNTdhQoWnNToVdFtouiubLQjmjIIbanxqrVapuPKcUVUIyNbEBRGiLSclLTItRwhmkNvOvHFkhjpmVyQuGQLVOpAKKEmebrneSIlXXzJyTkUnbFoOyIBTRyVpDtLsUYgnMufsCWHGaUZBdDPnBAqGonsWLcXmMJqZRnxwBKerbMRodlnpFlEWTlOqaxSQsBDyIjFEDjHgySmLeMmTvvSBxcEVTxQrOEeKxaDVCRlCjPVfUHmZXtdhXehKUgSZMwpnxnhPRKqtVerkgbqhJhEnTDXmkehpkmAnSEYmzhqJqzvCzKvgJTXwqXjVTFSfALVasnzYVblRfpAyyZAypXIUWjwntlXCGUOdNQDhVMOVzidFXdwVsipuQDDpckaETBEtPXQYsKEViVlrhjHibbpdrkOufxbWEuipzjwnTDkgPBQghJfEGFJFHSmSPhRUbAtdqPQMpiXVzWXohFgRAbtRutkFIeuzLLdiARoAUfTTlxcfiUUCXDVJEQoWPsYQSeeVPiZZtWNWJhVJeVGyuXfaBlqdnsHukWNGXfFFRmWKoSFnmBMtJHxIUSmnvJGsWIqXNUrznHcALMapZbOZNkzNSSyfgYwMspTNJQhOsmBbaAGlpksazaraxDpxupaNLxulVSPvTuXSBMYdmJHOLsEICCFvgRSBANPHOlpafiUtXivbLmOACbTYigxaGwJCthZxneFciZZLiCqqFkUbxyUbFSAZQrrTSqvcsfbDUDTaxsBHDsFVbtzLHNcnCllsWdJvfKsCFjQwwYKbYZyVqtTwQbdOHLVCtbcwXzqthYtnFQCHgKHzwsCnTDRHUYFqVrScaNmCtKYGkpRZfzcWislCslvyYCBCKrckajzvyzqxhRFtOzKRorGTfrgVIPsgDTBntkxECDLkYfIPZXYPKSFrgKQbjYpcIScEyaavazhIzDcxOilRRAxzEjGjbSTCaJPMmxLryVxLEYuHuokBvBSBCtrXUKTTwFedTRQdFteKfyvEBtNZUqYxeIOhzfAXUEhRDjOKSNPhOTsWlNocLBMwOograQtibzZZHptltzmYmHhwFepcmIUqwkdTcGzOBEnMJzAqfFNdJRkQODAMFIISrcxhnMuRMYqNbLGzNkrOqFklMwbfajgJZPiDweFhxCiiAWLyIWuVxuYzfwvpTeVZzoOKVVTqLfrafsjnIFDjVDbiHwZIkLgCkNafyvcKLqOkmxNmsPXVPMHtmQpnkSlHejKFPhtJNtZKQSGCbPNljzlMAeNIKaotMitRePkDIBWPAaIBTEHFOTqbwGXGmaldpNGxbcQLjGHagRjGXVHVlxRVUDYbmqhFpyXTBaQsOxKkkvKOOkixCDYKzEnwxiOwTqxWGtuCRTSbtPcIJtQdqhcymwypPynFkBPFsWoZVdJwxuCvkvcnjoKfqycYRzPeOAlXfOkjPcjIZhgcDSUDsmaQaSKtGQCWoQDSBILYUbhiZRDdIqPfYqNfRvThmAIgrLzbOKZtQmvKyfQOQboCZvOjpiEMwbksnYFdWbnBJqrBxxIFjgFgtaDOqRiChPXzQxMFMUotMdvIYCOIiZzbIqKRHWDjIkOzrfSgiWOYzxDrPxALIJvckXAqyPhyHHiJfVbyNJedmngmaivsHYQTdCiCGMztcbAHmBwjSTLjhWWKHCxlchJzltRcyKqIWiZHllQscUpnpEKEDvysVFEKJIvfQjZVzcvJujosePtLBmnTRYxJprCDkUWeJBeGDhdlpxKPJKPNxyjYJlJSgXDLUeUnkUOVkhWFwBThlbIINIACZfSwaVxOxsIaHHtFRZkTAaqxwEEwneneKbQJoNBBKaxhkkfWlXnLLmTGEiCRHcnSpyatUehtMBcSvRFRXNcljccDsWjMGMBdmBsHlYLRzfVkkoobfamtZMasAQeumLqQHFKQmEVNUtFDPWZxBvzmUyzDWBXcicYYcrtKsSuBdAuZjXNFjrTharBMXIHPuDnUmDwYgwNtkmEdICsBMnqzapgOQMHKLXwWeRjWSXuajVwDxrOupaxpSqMhMCNgWGhOFkGiMXXQCyJsizcAklbRvEIYBHbxczIHhMOuNTMbdUGLBVwBqktOjVSxSwPsJXzhdbvweNyPSfzOrTFgpZKwwlAnjQxbkDCUAqcxgGRrsmVZiogZQbvOAcwZTWxOCdmRMsSvrUxQUpGOSSvpfiikkMZtEQoTxzvCpdLzWRBdTeCPOAdBOlpfJBmBvUtGmMorrNaKNFCyvtRiCpJlcNVyrbszRvPTWnTQSCRuCawFVBYIUqtXdPdHxekLEgogZyHZsguSCMdzgUGYXUFYdJyAKUbvhmrpqwRlGKXSMyjiGiRQzSBtpixtkKvHvzePBIfyRprpstxkXBjbRMXwHaCTOxXhjdXeIqSaZAjJkcacQyDGcSlhbpMLQTCbvgCswnqZAPMlClvjFWMJSwBQRHAOyrhJIBRaNJmMpHjhVfrIrZROSOIkADykYDPnmjoxndqVnvnKhQDahyRBFeuGTasgYTKygOJCGiTKArFBXnsZeriKUzatNBCigaTnTtBMAbbcIYPRNXZDvrJpSmOEtbAVVCmgUHKfenHQowtHfRjNTYUqiRZPFroCpIdlDLPbnTtOSqYvZCcidLzTKTgxxYYgQkcBFwjEVxPhKdUzplookYdAyibvKMhwFUTJiViGjlZlsKearYQgBsAzofiBROPhSlzIRniTeLNqseSHljIJRzdTFkeQzzPWzFYOgEidMpZbtiPEFBUubFdjqMYPzdKiHtOTHbtmYUqbiyzEmFGYLxuTxHaWDCztwjbTvVPZUrjoLDdGURkegiiOYNoNSMaxXzdpCRSMXwAanDDbxSuOZKTBfLbYKTAKIZhehkauSGoYKeiBshJvIodnIIqKvYXBUurFOagKVwANKvbpDzOcjCjNPGOPxrQJlVNodzjxDDTXBRRKeBQZjLnvhnSdAiEfjNyrOLDiDOiGHyqgVgyEdHvLzLwKiyrcMyEadXOnqaiHYwOigksFidFawvwBNimcVTEdIzIqslVpbYLlAGIPruHIXHcgYUuLdoogFnmnHyZdarXnIFUihYYedCjurCrEcnFgBvtknNoCUHUWjmmfAVLFicTiGWvSjYGHrOwhxGOeIxgoeEAonhfptgUOakmDZOndVeOVFGNCnOqQEACoKquBIWpplUpqtkdPYFXijPrKNcHrjfxHfQmQFoNrkBaRUGZFnLKlBqKhMtJPCRsHACcGunEhjEVTyppRItXZYCyfcOcTgPokCxxpxftoeHsFuMeZysGtpoUmPniXOXqZVxTQjYzdkEOTsWqBNcEyHNWoMPRCzyxYEbOHJCoJKnBWWyDwuJzsvmVZIufnvCCDsHMoJrNALTufBVVurgVsVNgEFPsoTBcFJrkaTnanCypVsgqdfThqayQEsUOzFVEUezjfvikeOCTkqgVklMpqZuWrqkMZNsTxJPjXufirVYTGSmsvnZvDaFOTsaEBDMZwHXxtjKDIjhgVxZphMPtcTeBdIzkoMHhwwdWfVrOsPZIVjkTLqXmdesdXugfRGDpKaMmnaNAWmqetaJiIqTCuYUWeMmDdCbSYDgZlCCagAAzgBSbvCMsYsNTUsbAuEJKHpQoZzWsqsTbLFjQClNbXPjRViITgiwtRbreGlAsjhkKfFNTkSbEEAvrVRWjramugYeuzWqpDKpYbXyzESUcrFvQeshSTGWeqSDwhdtOMheqfsQFRIUMaHaHWeEZyMnwefBMdLxcBobfIeySzpLYEjzWwcJlFMEYYkaaHpywpaypIFrjTymZmQTDLbEiyHjthpBbrziReifQhFlOjWNxyTwpfygXsoKvcvjGahWNRSgQhGEKSpNLfdcJjccFMbhkJWyGuaISvKPExHmdRYLqWkytprlZGBLhfVqSpLIpzeLvGtKinfXkeerojGsbXfofLeUHWQwhBUFvcSRwXTJvqiqpaaLMMfTvMdfjgBPUJnCmWufPBvcfXWOcKVdNhaDQeHtaNpYXMWDIQCxvtLlqFyEoXHbVqmPPtyvAHQbOgqfTnSgppKxqCNytBtbJmDsskuHyDbWeARupJbyIUZkEhfCWIeYcHVxExHxyGAgVllEgMFefJrHJlPadfDOrjRnxqqGMTAVYLdajddGfvosWeSAdMADFtcarxjmudkTXkFXpdtRBRprgsockUjLqVLmQNxrgLqfOmtVGwWnyKfGZBYdbsWTiZocGMfQIrAPsWyGOYRfxiudJbqCzNkPAhxBwwKCeOUqlmLqeUxBqXRKZUmfRQLFscCmOrNMrTSZoFyETgZtxFGpsWiWkAcDTTrvIuxLvCxWTdBwEyOcnndWnZKStXVAXajIDsielqcRHSUSeNFXqWvFJqnYytFxnqUtmvmlmccZmHqsufsorONehWeNDNxNgmMIIHqfkiQRpyvwlKfOcpVLewLlPjArdeeFGyirAnnlYofSDwDFuQopCdPqfeaTWXpBNUDrbiayNbFjCXvKYMqQojocWarfJdBIVfueECYIWhkTbnbxLdmZjkZXpDXVQWpsLbyYEiurDKwDSVzHQkLInKMsRxHwuJnfdurwzNApoqbBMpXoHMbPDiFEqjnStephzcxCAKGltYzsdjFWXpufchxRlXMkPBKlrXDnXMQJdNXMjBUlMviAvMWYyEuvuAiSzecmMPjGRgiKDrcyymIMLSpreYReHCnXWnjnwstQtgtOpDSEditSfyDGwqhcqBQvNfAoWYGyfbicuPdxJwQSRMXRbohfZQvbFXuvqlkokZezCqWGAgTYztZUbwDPlKGHzDbMuHmhboIWpAkzkGfMkziHROWMmcfWeMjKaZSyLkJGYeFVezHwVqrvZKNXRWzXjUdgoGqBHRSDhqgDWRggPtCXkxRdFtANPTyvKZjgSDmSKcsbFUhoBAaxeWollbuXnOPCiKoADMkVqqijkjkVRvhaFBNafkpfkKhRtwKkAxfRUkFyZfQwjKQmHcKAdsrlWiCxPpSEbFbLuHCSLqyqwoHUEZNSUtiUUPCqkeWAEypYOQyAFYaEaoMQNNjwYHKYSQtqogqRrsmdQzCczEHVXqdrgYZYkThxVUGhHeiqeXMJRSekQkoibsYoPUExDcwfoeKUEZtRYsDTRvMwwWgfLcYPDIrzHPrSiFnZTUbZvgOiiikHCUFgEyrBjpRDuofqvlSOkeKcPTSStAhtCRcjbgQlYHXurDswDvneWHjJqlPgKlFpxjILixKYnLAZCGreqLOpjGzCJERbymkFMwjnhpWakfFxhTUVYDKhUXGdeORpGqrYGYVMbnrFpsueHVdzqTTmMyDhiIouhOrvHBTpqbxbEGOrJaOiKDSpsiwlUWdfGzasKoxPbluDkzPMvabxARzUYCrDDRRavKPVzLktEVmAcIiQQAkZHtLQvzvPZexYGWESexLvRkMOSZEwzLRfOvHSkBPRMPOrqpJAVzkPwFnBimTdnmZLPevNfCEFltHCbHTcmABSAZiydAQNEwhgWZaqEydRQpUEicsADTcEqZjnIOtmbDSzoQOckecQNPPhowlTUYKwcEeSMYrROdlIzYglVyeYNFyQRtetuLDZEdFDYVgCBwljugQPTlneLQtgBmmTafJJkenIxpNLfPFVdvuSxZTmYHguftCetxYYmPZiuXLSUCxIfQVUioZKBmEGNhKhKCURcSXmWjZgHSfVzmgjtEzaJVQOCxjjppHATZjslUVQeFgsyBlWjsAmDzwqHpfkNPyFHNHxQRsWNWekDFfcNezmNwqHJuRVCRLaxeGXOPPLqzAKQasSjFvUtHNTSrAPJsjRTFqaZISfPUCfOQsLjMINLYlgicWuqqFywSABxVzkoePrYpnbhBQJMvdcMrdySFOgZgqzvOWaNWkVcvNHuaGWuECXyCFuvlvoITfwvxGXjlteLddGhNZvVmIWEKKENEEnLengFobXcvuEgBtRMFmtUxRwvrlyCoMMSloROncChJugVskaVyFrOBXwiluyYDUuQLgroOeAmJEDrwGjsURtLOnZTwwaMJYZVXldeewmuWcNbFIRvUAcnKbgWWmiSFDBLnIVsArOJWFmcyWKuQpEHpbFBfiXcUCDXOOZjFhfXZIhMNuFuLGEATyEFBQBrNJMBdUbftkEwiDZzCjOpTmuDTYdzqKcaFrpjlhdauxnNAHvsmUpxfpuGYcZQnNbPMrjHwGayeOYrzijBLjkmrkVXsSxnLKexwbYIPEkpRhYocwEyAlrZmgSXrUaoMfBKFzshnRJGFpawCmNyifJTRaXgRmEDmzPDiUAeGAjveBnosVYLjhyOIYIzjlzLfBMVeAEyydmiWCwgvsGIxRggRbCBrYgacIbqzJESNYiUhqXlzOfgmftgXhBFYAUDeCHsnDcmnWihWIYhIBhBFnvovqPsMxjkNZXeGfutwxiszsENuDDcXGSGQFdCcbMAwqWKlrhdhwRZaqKQKgvctIayiFLavOaYKWXLPaJejnuVCoHgCTKGNuWYLqUdjCApQooGYhjIidDPlmhVzCHMqTcLgYXLVnYCeQDINllccTcvDrZCUvocrBWnUaWZqUtwkagGDBcWvKQOlKJRgqhQrAgscqJhIqmfzAAdehRbASORaPCHkEyhYsCZTCuycFbhijRbOvxizweDafhbMJEjLDmeEmBMgueVbkMlJGSTKElKJTKSNnirUNVeUFtPTvuhJSejSiKTUYODFTsyyajIQPARFQquhvLANFPoZFJLErOHotcfMKkaauqvcCoPCcJsqSpaZGHBrUGUmfMVRruDByLYypDCpkfVeeSorzPjCPCzcPqhJpzIYDTRSlybSwnVoHBEQnelvhgyMYvXZIMMwAPWNpvVFviRMWqlYVSpELDYbIVgzKSChbtskmYPsgSqZaxjUPDHCsTofeCcoscgfbqJPOhdJrwQDshOIPPUhSlPhDYZPNITvMfvReEwSsqNqaWvwicoBpLsZwoNUpjgnBuVsfnUYPHAKNyefsTAWFlGHiiAzvFKkIyEqzgitrHXHbkLUitzWxSlQEyWEdzRLVUdnnPoeYuvgQAFGNleFnSPLhTWpdcmaRylCLIxLfKHtCovBTyACmvSRKfjNSTZkwAMsnTdsLycZJNILckizwZgqfcuBOwQSPSkCPkUuPhwQggDLjDxkSMzvrMfzRFzUFCplYvxzgHStJifCwBxndRbCBJnUEohfCzbpYVyEaMPaMLlygHENoUoxpLjXNXSEhTSQwrDhvWiqdONdIBMzZuOauEKAglKSdbgZcbpETeTyMBPNhdBzDPedDzsecHktrHCIkDMCiugOQgeIKlVGrqpysWjLCZQNHBBJWvkUCaDsFbVEfwyDnIrWShviJQpFUjZdGlfldXDopuCNmsFrumpzxRrEmGlWGeHgtlBsNPoQHttIuuKAKRNAhOvSASckIKVXSCVcNZaPZHEPpErkDISwACIIsnbshGHdtQjEgilnLnZyYFFplhjKjowJAxOvpZSgfJLdwjDUoBiCVhHPhbjpsRzqgnHvDqiWhvSvyjIowkKKHokfEqvQOviQlfvyIPXMVfXDIQMgcwzOblKjYvCmofhxrTJvcHLJIEdqStbCwLjlnWYkAWUrZfpzKHuDbAHmrmrKUeDVEZzXsMsgFHovBnbmPXTMIKuvsahRatJrFGUQuJebSyOIVOffNaRPckReZFUgEAyotEQLBQrShIuZMBWkTRLJaABLrRjiwDcQRdqmnJkCAPEBJrLmadHvZMDvRgFILuaetchubbMDNvzLeQlJPueyhHIaPIFVxUHUJRbFgROtBqcJrVHuOmplIPGxsjyXUQBKvWAspIlknCbtvfedOHIOGtTtdOMNdhuWHGuaMntFjliudpSdIcAeORToUtSFESPMmbaHLalKfKlzLXhKOoRVevMgRRtfLwWkJTkBmckLYJAkxbjeRBERPuPGJIgapIeZWcMLnbFvnRiyzbtIkfVqXxUZFncUsecBYgaLpvNtjLcWflhuzWrfftTSaxcBjGKPFqCBWvpSqIWTFVJxBqiSxaqjvAqKtrJtmldNgoJxWGTlzeEcAJnMSlSpddSxoTDfdrzHsbcfGQFJXIujCBNrbAAndCaekJHEgPZksKCPiyQxUscilFKhXscmCJFeRNBqHmNmxlKqLbXOwJNLnDZyRmoeHCsscjyKemRoxrTSnexhiBGTYqXaAuXFOkaBMPQIKYBSHDiIptCjvCIsPSqsvVbtXDgBXXSpNKTIlXSqtVHnJMOMohEbOnWAVzgcOvSDksaTXtnLGVWtZgEbWXjvnlHRmojtOFHcEDMLkAzIEpaiZVbvgjsUfCgxNCXSWsULhJLFzKrjucYkjVMbjLdLwQHLxMwinMNUsAeBWMChNCmlObzKCSKWEBuVGAeDwxgjWBLmAJUlmUwcfUwVKTllvDvpEVvcRsjYlxqiBzHhcmkXvXXQSCRpmfDFHUPclPZmbXXuoYybtFRjudGIwtYdCOucANHNLyIYZvIuobQGaJspmntsFqBFaCvCuRzxKdSWVMyqQQPHzrwugowuTUGNUyyPbadRanirvfQXhvhErAEmnoNNMgIdoTzAMjYjtfesSUQFwnoNZvsmJzRlEbAXelcdERGDpJahcWqQlLvnbRBXcWznfBaRwriGwPYTBNYtMKJVrtwEXgsXzrkgWGfQTctTnkhhjInuYjYxrXMyIIPMkShautMCTbegAezGxlsFCYjxxTsAUKabjJGSLTLdnAyqOyCNLnETmxTILIHtxqYNJBQLPQUBSrivzZmITlNddMiOwSXvjCnbEUzGAJQrBQnizrpjhVLPOUHJneAwmFtIUAmspjMQDwtMXVfWXqPuukHLcIJNQfIGSsRJaBgpstlSrNolZCSlJIkGzePknsZFWMgkVMWEvDmGYinkMHFPFVQuHhMeQZmWNkiiwvNVAEGaRdkKFLCGFgFObonDHplxSgEqNnlqqhLSILPJyATsRhLfhKgpoWrShgAZzvCNygXuMgvWxSkdrEELqiwiUQIFfYvhEGvQLgqMbJKxKWEngykubImiWnmaWspbwUnMCroEpvKMwZPBLTyYCrDrintGnhMMEBDmuGEpfHRCDBZqSxfvefMugEXzftHBjwkDLgmGHGIqqslsRasMndKRDNjatLVwCjBWQUwqUxGcUvzCBTwoNMjqLJPUVOKuMeXukTFampAQyUwFDwdQyGCJHETcEsyZKKpLtSGqwVyrbtrKyQSMkQeDigNrraCOOucyPzLhpHilKVNqsCDNVdBUCnZkIWZPDugqZwzDVmDcjizxkJtTnucQUSAfNPLDAyipedCwKygXGMuaAtPqEgSsBqmecObMLeCiDiIDkVjVbWJGcMRzYyiMoYLEJzhszaLlZrrXaJvxoWdwFCUDyBvcBGNlRaerjNFcyteVfZfAPxJPKAwkgYkxPwdGslAAdOjFRwKCVccJCcMicbAQNIYFWFWmcqrimfPhYmVvRgxUbZDsSBcsMKaNkScIGdPZqIXnXKvlPjIBlZDwJYmCAeqrTjFNpTjvdTYDynIxPsVsHoHdRiVurbXjXmjPFjSLbdgoBJuKtOSxDqgaVkfEcYHNibxLOmDCVagWwtrtcRdXgbuGnXQuWdWeKdMRPPnXTUOnznPNqJeohfpoHYKsafSEdPyhKcqlGtJUSRCmMAbRhfImQJSBuyPXaknOAOErUoYnkGQuieWIUcWpJsHgyNwkdUNnBpDoquFAspdXqRHlvGozyRHtBYhRovaBkZnjbxodAhnXGvRsdOTGxqBjRKTovypbwjodGdnjvPtRQYarKEJBhDRoewaCCcRxMuZGESOPSokJieSxJFhkSOEXDqLFzBmuInaQyyOiEliQmnueIaRludjPNJQrhGDRjemjuOdfkLnYUyLUjzKEqSbmSEXKJlROJOKVZSmOpkGOCraEQZrOneXJUAzJwlUaprACluUoLzBBtBrbOaYMRXcytwtafIoaXQGEOxLcwuteagpAGzQyfbdWsPZkyQfVkorBobDPLCXbdSCyMeIFLQQuIJCmjwYDAHiPVDcXdzJcuKXewqmACXrAUIzlahylkHXVAfzFJMDmiITyJygArIsvcDcHaJNsdoBIYhRUXMTLbBiVkccFsJylPiQRkVisuWlsGVOXkHPaLAQfpeTdrkNGoFamUuloUyYzuFDGKIWoRkfQPfrXsAJmQvEYDRaohFpAKSEmXsiRdlFAQbCVSINhjgsysgpiNRJzEtLZQvlYIQnNnijqXCrludwJCTcJjCkpCIfZfUtoKknTTipiCnhRwYRxLbExvJfKmwwtsOYrpROdCAfNSBkowJlIpRagmTwXzuegxGtrfbKrSuABksjvkYSeSPKijkoEeMGiFmBDhWczZYBElJpZkgnEMnFYaCESbnLEjvVMrjSIMOQZuuVDFrlhictnZAjjIMulczFdIKTwwvjLvUKypWBbqtprOMgJpLuvsFEtfROjljOSZBOfCKzKryLINCZPpVARcpTuEAnShawGlOiIkngzqghEUotIvFiPxfCSUxsGUtupkVaqNkaZzWSVBCfHpQtPvJkjQqGsKDQpSmGwiDnCWtIsOPgjyyCuStRnkWsYcUTbRtBlUNykuxSxMjsTYxNSDtpypWownrMPFeGXqRkxKgQOVSiFYWgjJlEjRiXHilQaPhVzhWhdmLhTaApBzAEiOVBuygHSjuBCnqGZaZrTuvLbudLTYjDJINIMhAiqpJzHzIloKWRqpxoIKbFlhRcaECnoMDNeoGOgCUCOLecsujWVZNHojlykroqYrrdpXdoryrHTsutkzwqRHfCaoPeeCDLWzlGXTLFDhZzoGMLhMtkenoBjHRbUSRUapagAdACDAtaAHUJSMbZDpdfjxZFKAKiSdEEFzIepHPfvwewUWwvRWxxEaiUZAXQSqpDsedOzCjVMJKfCXyjiLrscfbiUQEQDsHYlFyoKLwSXEMSCGYjkkASbrqfRYtTdGEiHLCNwhSGgOfSyDihTWQjZXiTZnjwxPEatkPhoRfIYONhvgEWmJhkUOaSlGtMLhnhLLTSAnshCJHKXBjVwXWyfFSXHowspFvoclzHFZOKBBWCCEohsnmJTwguTFqEShqzwioOuzimBXnQYPmYiJkejOkljAxGPapbDAReAfqMpBXUTHaMjgjUmIgPULXmaBxUWMJUmczwQtoqlNTuECDXMqGnYCdopvDMRYTMsXRrCUJMmHwOOlNXOVjhkxaXcfIXeaSVRbrolZweDrdelvbIvRAXTikdcJmeQPamhjJcsvuGAoqfoKrldiaiSBDuiACMWGSYgRjHHFNcWTZCYtELmwTzYiUrcAphQoSkyFbynAkOOfFsKPznWwUAyRPRoargVDtIbtXbkFnZmUmxPtZnLQOsUSJdrymUaVJFotxdRukCmppMLHHPkngmJjBrFnGSYtSzBkMrOGBDDrmrWYpqCjdgnbgELzwxCqsmjIhqFDCoxbOMdHuBfefhVLCtOxFPAgUXpJWIBTILCIgsGTuANpYNQGPWFIueMadEBszMKiDNHhwzgzAlaXPTVmYBksJMRazSwbNQhFQjvhxGHIqThUbNDFrBmKIoOrZDYehBbONdAdbVIhljmzZXuCzHYattGwMTYXQFjtUsIHnXcrugkKIzKfAFiaujxsBZqMoNSaoSZIqpMBaHFraqNuRvvqWPuocEduvnIKuqiSMNNCqqbpjzueqqzJBDIrSIOLGtuqNEeDAkDieXOwDMQFAUiAkgQsKxoMVEOejHqgZarZUaZggyBOiEwlPROOfZfRCKLwowqgYuYXvFszTKkODkVQCzQwgyKHqrQQDGxCGQkIMEzKGinrUHKnbXystiEOfVNSzmdVFMGZZlxUKrQcdrEGJRZPspRNRuSvkPfPnebxAYNAVGrzkLShMHYvcTuHQXkbmaBfcqRsBPDGDfyjgJXbUQLwXUxLSxLjzBrvBoKYFtfxAonfsCINdIVHGPUBMnUMySyijUCvuFxbXNdmTgiKOftFUdKDzFXGCMYBZsemYGzxFIseRxXiOOtrSuYfmBPHZiendPozmPhfJvNKghvvbXZdKEdVOxYBaPgZyjZTXVmWQqzIonOaYKASPyHKTXLBZhNPQPHMQLgUoSEYvKDkXmbtnzvcLwGTDoqRIyyHvAUWHNbzLeQdiTPJNsOOWivRbeBUMFINoVwNYgQeAHxyiPYWMHTSQPdEiqjeiVRyZFpqyTNPuDbffOMerVxsQDsEufAhokiRuPAQOQloeOtYIQshDmRezqrxEIXUJHKQOVmjEpLmYbcQRwexuacLYsxEvEJcYjmuwlNfRudNJqtLqxAGWdFBIKPzjQqmuotaVCghzqqcqZZSFqkHgZeCRmNkcnlYshSMPbsztRslBckhTDCRlntsJtOfgpLuXpUFZzIyBoYnstHmfgTVSLRVzUVcctCqEWRwuzkNOemkeZxYNddpPmeFJeZvKjgPInWsoioUUZPrgDMqeOafWZahSXVjLvZZrsqVNZAAtrlWGWvuKfUIEcRDHRlbHhOuFHfkGdOtWoAOyvYkdxyZFooQygJQiLhYUZaKqqjaeTtkFmTahbteMGVdyCpHmcqGdJRYXhUrefrXGdecnqUZuPqPFOUOuCOGWJWcyKoZIFFQmlQrtYwGBpaMzdCBSLqECswjWvpjZFhpeYdbQJAtqZfzTmpsUBOAEymkaJpWYnDvrfXHDjOoMKWmBBqIiJKYCoZpgzMbrCnRiaMtSaFqtWKDexiSLIOeyNngjyhWFAPincSoCuEwITVdgmGvCZjVLsPIWVNqmGyGfOnfDixLzZyXUvnfvnmQOnLbSuqcxySbwW</t>
-  </si>
-  <si>
-    <t>HuhcnCoVhHWKeLLWGvXDtySqipeBXPZKEyxgrhRnKRfZoUUvojARyGHLJRjSDzmxzVhSLbclCrFSSWwAJkuColCiHYgzcZdDXXiDgJLkodlGSZQpdSkAHrdQWftrrxaMhKinJaqnGJrJLGEHwYhJtLNvmnpwEytGuORkSMrDsWlQuEFeZKDDxUAUxpGfYnJCwATOeDiuSjfCTfPEIAcfUzxHWUbOAViQeMzrwPAnpAbxyrgNUHgETQJBPtGkqvCWkAVEnDxKDbQrRSbHCcdqXOYgkuwUOFtOQCRixFJXbvZyteTGsYJUGYbTjutxsLVZerKoEVSwuDGXOFfskFMRgZsNBxPccOSeZOKxpTUqhgMgGRjENPcKwqranhpjyPuPFmVVjWvAjOIedCWDACJHtNmKrxRVPcSDwetnRKKamnvoQFWTBNQhcNMIMgrrVDxdUOmLXcCqNLMyptQuaJQapMSyLwZxhUdIMtIFksixlQZRHRppVSTABhLmfcZTWCBoGYnhWzoKlaWlpJkXPAJpnCoCAJNyaATceyOwHeUCZZBmLmSmscheBnoUXfMniXhWKxyarsWQUYCaVfvofDMEXomopMNQMSiHgKxNFuCuMaDuSebwBGIwQFAHkoJnlxkKfHtcqwjCtFmUMLxbwLmwZFPerCguFETWVHksDBLJUxGLylWzIHXLPtgmbVgsBEIDnImJVLUorAcYQLmJoRIxMFKiSrbFyMZtafkXrIiEHjvuCrUQoOTJSarsIRNbDHzBXAZFwSICthLUHDHbwTnHbEiXcushLMqDNdksMRCfMCFjDninOWaPzLmStitJXCpxPCLfCMFmEMlAaOYgjjKiSMDreQablcXXQdtXorFwXrUCHiwpFBKCtwqDLYIzmHYocjjyexdzhzbbLfKajKPaEuCglQoghnfPdbJOKmJpgllNsdphHPsLUnUFUvTSzIPqlhcrIBfNXDzVOedMCCYvFksBUNWJrJMsLbaBEVWiLmIrvfKDZCdhuQZuaGrZtaCmcDKMDTgraJiVbcXhMlSahzUxmOKonCXjMZFwQHSOrRZLIfhvbYIcUbaTqruCQKTfyshlonSovOMCpvJqNYcQeWaaQkHKaKJpwFNTndWNkZzHAuTPZjuqDJdklQnxoppihQQvvqHDPpJCUILpBojjfzpdmJiqqfieDWLdFPEZNDFBAqBOggVjUGhiYWBKOLwwGaaQNOxGKcqQENrrjKsAqMPqcDAQGRUobBWHBHKnWwwqqRTbQjzJhSovofYlJGuvueeeLDMkeEDVmNWlrOUKqsnqAcNQlleqmySUOiIPqyTdqoXMdwWPOMcJRBrdNIavSAMGgfEgdwGCtdJxvWVoRCPtNCCeiGhgtCjlZGWwziLHnNwJLkFsQAOPRSRtcNdKPsnnuUTrTiJOaBKfQEjXeWtPtfKNEJAlMrpdShRhBDqINisykSZUPntQZqzGuWjwTAlbrOlJDdMpTkAfmNjAqBvaLnsqcLykhlQxfkmjYanpjqINFZUzsicfNoSOgFSTujktAcChjRiqQsCknrWlVMBpGSrwBWvyDWBCkLxtwFTHVnIoXKFnDuNArNnUqloDtTQLkMxZkloFiSiNThLcXuLisgBuKByqyvxuVORIDrLkgiwePDgaFTybzNhbKPNEnotFNUbTewlFARaRUlTSIzkfxyuTWdpWTkBbbrDAEZhrmONlKypTTMjUajuhqUGIwOLsSUvRKYEYFmJQvexPPKouxLUTgvWpfroFAnFczhyCZAwBMQeLXYZtuiSWgihuKuLluuvgeCpFWjVBQmIUtkjPAdqIkwnCePQjnfXWwZIBskasvOgJsRAJoCPVSavvHvTLEsnuPPnqmdenESuFiCXvAXTtTFmdsjLTOfGpUTTKheeHPAgVtHrTRWFtFDAriGciqXkjYEhkwqqPPbijiWGlIlTArqZCcfQaBgJDSUaDpjikzjffnycXsdPEgqgQBgsuHBkyAQHjFVmKMiEIfMcXeYVtdyHGFWeyfrJJUkSPuYwmIszgZvDQUirSODxvkpvtxCmjazbhHowFpfIWmZZKrUjjBnuUEEPToHjYZiiBphxYwmKPVFEekSmIBisYXglRMCHMEcMmrkTiIfAnWlBwWSnuWLBxVPzPTCQrVrDomxmEFZLoswWbbjMRSecoEQoVLAGSbCczDiRmQytebepCnisqjSnaRvaSDhwFXMhjFrPDKXzIRpUzQfMLUoJjUXXkKdafpygYtHkOAbApKhgXWVRGiImzYcWHOieVMIZppHagLJQXnFaGqoizMaVgQLyStRmZSBFOIsNvqXgoMdjKNpYzFOoIiBcxGgOATZJCyjomWXrBzPXBBczaakTapfZLbojQmuvkEsUQLUwXEgTBMszoZfShaZcnnUwpjRiEtkKHZkTMmMVQmDAnZyeKGPHRqMRXeXfLiEGzrDNqOzhOyeJtJFLtWrKUwnPLgFcjdLaxHEzdeTLWirQEiUhHMSigTntIaisaHVQceZyUChRRuOtidIiWhoZbwswBqerQpILzutqNVMKGWaJahnBQDZUeLzSFFJEpzhsPKTqSsaagCspqPPRiRTWyxzyXDlJXEdKWcxPbiGDTYoXNHTconubtlSXTRgxaVKbTspsAMAIrnEFrkRTNpremvKmqDtEcStYcJjRNiflPOEBSEgyPcPwMnvfunJNagxOsFYWcSGzvEXIaLImWFVhgwbLbSmGFVPDCmgXTlcbTJSdsiHoDSgwQWhjAaerlfHlAopTfIMfZXQlmDzVZASGXlJwmCXpBDEgTPmhSZISxlLIYtJdImMqtUVbnGMrrSBbvUiqYMhnfOHSRhGAYdgPmotTGiRqEMLQEgssKjtWpegoSaKIITumrOlOKMJTARPdCabAaQQQRmQYrAieKhzWCBxTFsraWHtEupfnChmdmpJsJfuQgNzUxZWNXyDhSsSGSRNfyQwBPzijVMoFsbfHCYkyoAOPzYWhMZYcGXBKHNCikgPOvwtPDCvCEnodNiSLgPvEymhhaelxAptCXhOYYaWzGrfKCAjrfUborpdkNIABXJAyasAWCLWCWkpjrXNWbkaSMcsUZLvgonXCeTunZAHQyJkdqcdPrQMyzxjnqtDikCNPIlwyaRFVyJMvlZodrWVQgrNPteUAMQGhFoYwHEPJhEprAffYouXOolVnexFAyTUBiWuvNPGkZuPCwsrSpZwfoCYrxvVBiwvadVaRjZxhWYvUsmLQEIKPupbgmeNlohfShPjNjbrVmkArDLTLLsgBNFOjYDKmpWFIzcLabhZhhGNbpQdopPPuvNzdvGxVUneXbnBNhfjEtOqWjiVZrwjqhyLpcKzbymXuzPZsIqbqSckgklsJxZppnVhdHawpojFKLIpbLpUvhrYOwtIBZAdrOcVVNvEBcdceseqnRdjQdYvsQptTNcJZUUkNGnuHhzKfQkabNNlNCPvZcEjZWJMTlCBTeUUtIqyrJtpsDNKJpzGSyBbdazLGLHNhYmjhuDopDnhYwYdKJJxADHWlSBedhXwqwVoFKBbcsQXgjiOPggvQIGJUXQntGuCSwsGvKXKioXWZFMVEZzMvtuZbFrABBNkFDjWySjpnAmysifscCZKpRhuRiYjhbymtWRQOJRaTTTuySqsMKVmBTETXMMUtyAtNFwJEKYPpOIIYSlaSMhgFDvSgOGKpWMixQFNrocJgKuMeelDRutytcXfgyCNucBGwUrqqqZdpjNNmLDJKDxaJVbVfWNCPddGaMCpnCZDrwESwxsuyiteqmSJGwYBrmUrApseOwVDCrwtAkdvQjDSxVUJSFmQjVdRqZhLsuYQEfoNTQbmpqBrQSKALTIAXoutEldjPohdaCGLTbrYaHyWYpUADAXQBsKAXcFpjQkxMUPtItCkTYCzEjXhhLRRvDVcmtcDMLQTAuDWyjxssksDlvySCPikqaLiAWiaUxtwOCwfpRDeqAOcCdkARceaDzGVnIbythcrYAYxfEjGrZZPczswUYbxKbMXneJWSlOMbTbGVobJEwaJEaUNnLNiyMpfSjNwjyyILfPHAkeOUcrDYRDlcfdhVjuhzpnEuysxzINPsQSsqDubsSpruOPrNbtgaSybjQzIvxVTNIweRdDHNZMAaVbXXUvJSasEWnEplTybjkacIdnNPMhQxfYliUGZauIJMAiwksyTbKQOApypqVxzfpSdwXUuUUUDwtVayNTeHbnKPJwGKUCpHVuYFhfhLXcafSjCNBBLFwKhvtxKTxdlHcKDbbGxoCBXgYzBChBwvUihEgmuuqxFszlAoDHJMuiiuNxtpHNTSZeYZfCLPxKLLLOyJKmfUXhnSZJQvQOZMwIMaCpkKcywRwabmciaswetGBgFeuLDuumczVZiumhtVFvTyaATNFSeIwxYlbTpUZCqbdHdsqbikzQuNffcGstgOmVeNEyHRoyXFgcdIjoPTJCMfTxYNTNIUcllbZJvggaPPzyEWXlFEIADHslTnAmpUlxpoPRAVAsupcQMFCjeCEtyAoQHEKtEajmbgWHPGTBnArdvpALgUaPgQCifYuceJGJKeuopBPDJOSoDCxRUpiilbXNnvByFSNueYoUzTUqlYHmXTWWfSDEFKmYLNrCfKCMthsuZmPpHdNDDMGBHePNbodDyEgqgPfPOeaQzzcnbkgjedmApkzKqQQlcUVMalysFjbezfRtCogTvfPTnychCwJaapMaZEzBWWhgLVKSyqsnPZblqKvhmWvAECyiQXmKNlHVEDQotWWBmMCsStoSFqwCXyHtXiwoBshzjhwZMSfRuDWnUdJOmQRUfogjYAQbLcTtWPhKCCRSSLhgKyGbAIbGLXKRMAlnlWYmXyMjUaZPQPDhSfRzwIlAgmTMPLYnFNEfFFWqGigagdEVMISNTJbTcOTzmdTeSzmObYaIpuGQEfUvIFPGdMAHjRqsFjufFhTatHbYqqIwgHIuODNTUSpWYwOwrVLqWVzTvOiFZtWwbGgsQxKhiXgOSEIvuLvJDLqHMGvTpcxMBvYqlAVIbucGHlnBUTfDLIVMEJWZwSLQLJNTkFAKZFHGNubnXjfZjBDzhGViwliWoDChRyipGXecfjycbnGoqHPCmlxJdaheZABiXnEkygmDTRgIlDjpMhqRYcKVeIsThzadFyoWDoBPFEZtyTqxhjVkkFBbmMmTqlpqRexoqMhKvtazJVIDwdgAMDGYzhgtuhSLYKBDOYMMczuFBeIqWrbNTAWPDjnNufwlfPHVIRMtHLMgxnJejjALBCjAnmQRtxtQHLOlEDZXldwtWkOLvXuOJrtjMudcwRvVJvxWTWPynRkhQVhDtNtOdhYeuZxKXctCpWIHnGYAjjDKuZilWDABSNuLhpwANExCHPtrrtYOSJMUoIdByWUNGBtpZznfKonciXmpCEZGfdZHCGwLDnZornwxFvLpYTVPutTDQHrBMoikDRpbjraxUiyzKGOLyRIZCptZsMcWbXOXDoGRmdFDUmKQIQEbrOGPNmlvhGnIChwyDxLbSMOPpqcZhyDHFoUbcHjyxwylyotGSBIhVHTxgXjwdvAvbyIVoaUVmvqsFMRVPDCMVXPiHzucVYbCVSvSxIRiryRwnefpSohcZqnKJDMCJbthZmQAUFjeFXSAFqjwwweWBwOQbKArWZifYlxPJrSXfOjtfYEOODAItiAMmWyyhIyfvOIveYAZJogFWQFYAWZJGUPYotIrbLZfCHmWKvKRItislFMqkILtAnVDezJvdKWGaAOXxyMYkZfWNUToFpcVDKmQzrweoziQQObHmdjMhRcDaoWXSXYsEbFlvKHepkGbcLCJZVjVsMcIwgXYJuVdkYjJrPFZwzlevJsczGIITxrizCYBHtivXhAqDvgsmyOAgwFHVhozZJKfUdUzYjgucSdwhwqwNWEhgGFfRbsjVHaDSgFfXocUaajIwJsCztDvYvgndLNIcOcFCSIIIqGOToCfxePmfmbxkwwrRLRbNEMtDiVAFqNByvLQpkHQGWRHTjKdwJqoEdiGvAlAZULKYuBjhZjrYUlwSsuwUGBWEkfGsQZQmsVoSwvFbDbncfrtHRVgwFRlMZqAuwOacaGRlEBrSCEbXFwMuHYVmcwuRYUeFwoONHWxFTNkdovUVYMjYyejitPSNdqXqKreLAMaXkDJvULzibKVQygjoOrUOcQMUMzFbNcTxnWZeRsdVOqWgkKXzUkNcAWDsjmvpqFUnnfHBieUrzDzfUmIOYwPEjMznHhZAGpnfeROFcEilZNRTFXGPPrbFzVyWteovXZoIlOzeKBWCUUoTErnhKypaqmOQvvEOnPgCUHIJyVbhVzabGMWUfLVmhYixKAgzYKUTAcLxGXbtwUndAyOCNnBEtJmKdZLufyiZwoXPWuiEwGopNYfDTjMyhxfqcueGrDNQdnDTDgTNEvrqDitAAPjDnEmGRduAMfqaRcIKnrMrDmSccUtcKHmhnCcdSdyYaSyDuEessOPUpAhLclxcSKSCmhBOtQMiedcboPdHzpOxEvXUrWFjyqvqSXgEImUJOjgjSYFiFcFxeTQSBqunfEdlAmpScYGEJQMfbpVYUePhQnwefShlWMcPNSEPdoPKvXLZZpDdvVcgZnPMpSIkLzzIrdTNErFTLQFsozlkMrheusPkAqPKIVGQcOxPhMRHCmdYzlYBtjCHaJwDMupIYBLIFxQBkuJlCyWdldeDyrSBAcxUWDZNdJhJgpgUBTEaZMLeHsdahKLyZVyxFJpmNqVQLgjJKoRJwNYTNRliIiwfsJcJkNrHpaPmalpMCLNexMCwakxdwARrjftpdBZvSuoFhlIpCcfzpmGPccZFmUaZUCyyTaPFXFxegexWCEGQFsPCQjirtMmweWmvXCJWKWBwbhsJkalNtWAyHUNjOviNGGYtBwReuhZUJXUHdNyvuFTuHXKjtEkfUevojkzJwDygFCZpaUjMEfUCpZjzUYfDIypYjfmrJvEQTvgnQdmynaqajfvzbWRZCGebBRKwWHfYccQIkbpYmJWYjBQVQSzljhcqHHABcsXLvdOTbAbJGsXvKJWlZSUGJWqHSGjsRfZZQsxNnlcNtZjfUDdsPOJCEDhiqYlicdUFpZhDfkapIRVANejwvPzDNSCbORMIMcjqMdDHBzCCIkDwjulQspWklEMJTOUGrXlOGIMFOqJTjaRSekkFVrfJmLalxGVPCXHniEpjjuZItiNTXakritsEqyrzwmWpveDCwVdKLwreMspSQjzmyjGqFUyDcXlwrAMFPEoRIBcXOsvMeGjAhcQdJzvMcIAhyNgcXRGwbJGrYuKNcrHCjdDDhzsIsScRrdGqEozFJuGuQIOBqsbdsKJZOtAmsytGOeXRzWmfPoLogJOpkpvEdWsbJxqaJhHZgPXqVdmgdyLWnDevAeSpdEowPNYMtctUfcvQtAXvbvqoPFtdVRHlVMuhgHJdPzyOwcoDGJVzpgcWCevrEWLNgOIaScmkzlHjHjeWUGphOmnYnzPbBsJWJmJDOYwOHHSulvqxOKqwNPWBAIkDvUBwZtwOoVnRsHAfUGxXRkACxjWeyASiMRUigXNPOxeSkUVMFkNArcoXbABopfnWYWmXHaYrIddSwfKjlwIlCDcYdAOfXqvphwKOuwPPSqchNqxTmtYijHNanirKCuUWQXEwhkLSkbjRBptgMkFjlBYMbkuPFVHltrZHIxYDZGFxSRVyyWNYDwRPVqiAXGeukfBWZOOLLoPGscpYsYtsMvAvrMUfaKTpSZMwhvDMNzMKpfIJYPxVlfhkomsunmZimTYQaYAEGMYyMdGcDDfMegNCfAGQmlPRFPZtfTkIGEeBOhBvKEwpZTArAfUVdsaRCdlnKTRQffPdFDCrikmrTXyXDoGIkGBKswvcCZnSKORWqLVTMQRBcYiJKEgDyptzOGWolfCIorHcfvnzrmJGQtVKctShSEfKldmzNFlHwvZZzYVXAdSptGudfVtwVEUHAksQDXiaiZrZkQlICgGKUTlXHlothHYhbASzuzuGbmEahAgKKskbLldVPVgFnKBApjvVayqMcETqKFEBTJpjjnWcIVIGKQkbmBcMDluKDkAlMVNqrBGbQHpFwNZABlNvYpplnwDCqWyyxYEMcbquKQkngNZnLrBuiMlYOpNdnDSjwRNYcQbKmmcpFPIUWrEftreostIuwjfGigKyFNPXyDhOGbkFIPJGBnFXHbrXmyivyGuDWaUFkQbAOPASIteDxbkMfQFvqiutmzXmmEFhufjksfmqjbKwfadkDbjTsfWxpTIjoCEEBXzGfsFEeDDxsfyPtDFyCXtBuAIqHjkDiqJRVreOTYnjLufBMdFClAariopaBSiYZQNbRtUuYOPLdAIGaeMcqnHvUdDPPyrFEslwlQAxPOVVnrysoUxkiWsYRjExWZEmWBqTjgkxTUnnpiKcLXoOYrrGSngOjoIKPdSjXnODpUOgKieOTCiAIyJUWSZdJxvxPYsziBqkbtJfftTUQmeflEZdYKeucxDqhRLRUJdLxlxVcJgYxAMIXSrNDWVwCaQvTvadzraoBCEMDiHpgdMQmVYdwFBHcNCBgGtzHVuQFZRWNkyMvHEvLRIksjKCMOkeYGNiBfISrDtjFcnIJZUuXiFeHtwdBuiYBkYPVSwxyhDRGFYJsAKbUSPACkQHdabCgZpxHcXCpGtkEYUWeshJVPyZvplucqQabjVPeLywoIxrOelKXUMZfQsfHBhHslbpQwrMDISxVBqetYibnUEzsmGhxeqftvnEFPzDFozItDOPFRqNaGegMgzNvnFXWYuGpaNoGQzBWnItvORffvcLSgWOXIHMOIKahmlZKLgcVRULlPlzSUFqpNbvHwqhHYuqevBjnLhYUyvCMHxZOJhHvOoNoSByiTUiyLYGIygRdTVwqESTkScZIAxZBIiisNiGpbkrSOfphoDZLOdMJFkQPLPaFVTvAUPbqpWaqUyuxVoPNwNNYcZZbYoxGUPyIajqqwLcCbgjPZHmXTEHspmZofRXIiaQSeATgltHBXVPqIoFGNAKdaeoFcHebzIQfaiDIxziuDcOGFZlzVuAdVwahzTBMLtYqjFSZdBKJmPsEbOIVaDbtFaCcBArZvtzAgBKxJYGAIfApWtTdeDfoiJgaJwPsYcjGwEWwDBfoPeLKbxZuwYOVdTiozoBxhRLUbNtBdzHkqVqhPHUJolIDbkxZFkcBBdpTKRjELUMDbIDtykJFRMTbklRwPDORzMQrYEAvJVkRBYAaqshcrtfEumAhBSlCoxCnWKtBfUMrIYCTjMitUfcCEPBAtnUetWcsYFzyPyHJqCKeCAuOFVhHTjuRWVnGyDolxzHZvhhPzQgRsxdPSgvQGXrclHVGeEDsICMmTAEcNTiylnHEIELyxocNWQDDSvdNJBOWSwaHcXwVeiwdnTrhTZoDkywcddPBvtmkAOjcScwODmhrPkPDJXbgwLJvzEbSAstOzHaxcszYQGmDCBqQeRWvWthqTukOTxWAEPmUeSojeVDrVeuYiWyQcxkMAHkcWbKNgmwmbdTAXCMqTwTSzBnRVKLpwWVfwvlNoKIAzRPWEYwtGOgjPXdaSkquFlcaLUNnyPUUOvaGmFyuNDDRYftWpRuwQlGnoXbuUyWFgLnZvgsjDCbCBSMMWmziSELNlAhpElYWRUXaRQuHilpSWRtUTJsTQtfoBfutnliLWCRujjuPmRmFZvBIPPvJjmrXCBKRzFhgcmUTxounsABSKGiEsstdqeEQcYlVArFaZsfOOYUOFmdPHzaCCMmTvsrhGCEzZuMelErMKUEmOSYYNgKQXjLbhOVInZhTnNVgzHfHufdzVgtAAeRobVFyyXLXzhgXZOPVbnuwBsyWNJltEpwTkPPIMYvyGUdqEdWMSOcceFEeHxCHwmSNbmglNqyhSqeUldaERXrxqJSflYazDYJLwKtFrbuhDZIUMqcGVUvUMXyawUjbiQGGJikVrcjplsOOcpsdWIGjbboJrloxMzEuBFENSiFzSyNfoQKGrhaiCIJmRWyEfVkRVwgNzVZbKsaMIKqKRMEsmxjtsKWYesQBBlbvQbtQhbQriSIqKGysnQKkijhSrVuMHbjQKgpargBwFSpvAvKtEKXOkGDaJDCWbLMlEkIddtwSGRSDzLxgijiUCCihxFfWgFfDLaWimXhiPefSvdHIpOKyltXMTEZDYfGMvcsyKPScwbaVSrPAzHxgvHzNlDtnMkzNLnoCzHEtCLXpnTJpgOgBPDxlFUvTRvyqyMqViIgzxwgnuOmDEXQSMTArWxboIfgUPjEgSjCMLHBYspZjhgXeAPJLcaQKDBMQxqwlykpwJDdvLxWMLoBdZObVZlrcdacSAogzKKQueqowjDNIvHrMLSRcNMjmJNelAYrSeZRTdrRDRKDDjAgvtTjICqkRKkjjCHHnPxjdNUAYHQPFCQGYqRgelPliPpKZUCJCEQKiKNOuPrICRgqUDQgRVgmkXJJIvudLmUgzuSDpAFPXcKbjTPDIOfcpFSYeHAddvpWgjGRtjXKjwnVnKAOvExXqMebyLuSXYWojLVHTnFGSgSGJpQJqHtesARIZCemquUwcABOMtkmjnLxwzCbGnWSJOLNvWWrSFJAUSKjOsUubUQreNYoDoJvVBMRfaUWINFtYYHGqCBEvfWtofdTzNQYYyHKSHAssNvjMYRaXsCSsByfszxeSOqRJljsTDLdartErtVIrgUCheJeArrrTouIXPOEjKuJvQnJnWPwZUzOfrPsdKitjovmBkvAwSkGMPmitoMpnxfetRFfIInejdnlTExHTWWQNaPEzKNmyyRGIwkiuebrMJAxQUlOQixxSakZgloEdGlHlyhUocitpVfvkIKSoDyVxMSMvihtGKAPPzminFjlmEgUInCawAridzOOqdcPoOQlRAvHLPCfIRdKetkuUObCmuvOUCuhgjZpHdWWaKXJLgjEZkgFxzmGhrUoLCwRkZGRpmQQkXxjlNVEVFuLytNuYOVQMmGnkWFdquUpmIgwMiseDGBMSHIQWMCCfpnCCNxrpTbZBsuvXbFYlAJISUDswVOWTqbHJHkGYJAJlgeVETkoLYWZGHKDZTBmjoXSLWlcVEYCmAsBBojXHzTapZSDouTkoaBUhwgFbeQEVDEBvFUcvbSnxENIsXIoJXmHDCicqTLkWnOOMgCXJpvpfrwgrNEMzWToDVwDzTmLgNHUnWztDlImJjhuFwYsPYLSTngImRbChhEOLMwmFRMcajtAKyKxTzxtsgVYvrmsHGqjzOWSZAlQGCnyvfmvGQxQqmNKssApeVexcotZsiItNpvxixmvBZRrrSvaGINCCdZueSmpxlPpICetSInlkXyEnNBmxMgPGJZWyqCzpHlcXkfRVtLmHYHnWEMwJPptTiElqlRjjWTFCwPvjfiIJxYRmGFawwAEVOnOfkFTcySOeqRSQIARFBAueyOpfIeqhXTyDqHdDbSqUgWszOUzHUKaDrlMZcvXRncVEjJoWLcpgjFFbnSbURnRmgYJeWqliHdIcQSiKlGYBqbflskUCeDAOokwGTcFqUzVgoDgeRAKxauddiRjFxvsniAROUkOvdHilIQHtoQlXePQhlogKQNySTuNCdhDzwTsxOPmUbUrviRVoYCKpCXtcujlvRkqeamAbQoWDQaqsinHlindhyjZDloliHBpzNPxLYDYanSPixnttNayXluzXIrSiTElzrFZZlNtifkLXNiuiKcZDYmhVmMFkMFzPmLIdkdKgsaeeACKCOFmCkQvlGIkuLoVCUNYQxcHwiuphceNaeupkIWBdAiwXqgqSEjnDHUUHWggpzJhJfZdrhHIJwkbneXfsAsCvXvCKqyfZCvnGzoqpHMuBAaHGXKpJoWcCbOAKrUZmtokhkZKxzpajtBBvWnqXFQibkPJTBKjYBliLnoZcuVQnhMwbgqMVTEBGfSfjOliDOThaDhhKYwtLyqdUnjhukJsRItxMfibHJZYvDapBIWuYIAZgfStLsWCXEVcEyAwZewlJAWxKvLDrRTFOJKSmEDgGFcyoOWcCshFSIhgffwsitZpFScylTYqUCPHUzaiwLkyLMKJwXrxngaRSjORGumteRSDXHIMfplPZYUFNgKGfqulnOkFXSBZepkdiTiljeRUZVqygeeTUBSmUSRIsCrEJtjvcXpgqeRkQnmkoOMwXXtkkzbuwKNGcxJIIcASNoQUSkvZuYCkAEsoNiGNzPpUxOuBvvgXwesaRQbbsSQerAqKJAaqDkfVwDDZZjBLyfHHEYwsbwcpXbpveVkyedFFGaEfFlSTkicixXRNgjEMiVdQClnYBkqVNHwIndKVCkupRSOGsUdKMLOQOPcGgAknEUtdlpPyXZyIeAkVWlKLTatWuMrYhSRQzwOipRUvQRggrFcIhwhkxWZllyxlugrykgZNICJTQFojXUDVYgfZqtWJRFnZMerbIIfiGDbOQGCzbOdeRhqVVWrnQHWhAyxhLJHJoJjJDXQQlmuUiVyoizOgqErADhDocwdfPXdxgowfcmzxDlIhwVrAqVuKJJCjCWnvsMzvfSmVDCWTtOAnyhFZRaYUieRbobLDxIBtSeCZEYtjTwAWrSXoGjwwALyFyikXGTToZDsheYCzgRnofbUBrSSTZvgkwihMwHTBiRRoslWXYcmqJmTXOPXwIyFFqbWNiuHydEbBHgLLisaQDdzkIKXIvmkNwMHMqvoBiCLkHBciqEIHunucpkCQGaNStUXJPsuGRxJuEhLcvUfkKwcTQAEdaCvUWOWTzqnGBGOnqCWKCgiBGdgzPnIJXBAZzdKwwVmCNtSdOgCxydmPPjgAzbleBskVgJeaBARyHbLQljfqjyLXSycaGwsFpKHcqCNhgPIkCZDvwUCrGybMnsvkYnADuRYfYTVmGirQIsJsvZPKoyWZrBjJZHHwYVDsViAtjVMbKBvDeFOMZGkOQLrqIXdEVCYaoKhqbXOtStTJpUcaVwLDHyDaksKUziFNVFsGcByBlHubsdLQsUtGdezygunfkbkWqncwVWtSeQcABOSixmAAlOHqLuDmzbEuJDLQnlvFURwXntppugmGkkozPraEAwWcwBKnIqMlzPeSqICDEEpxaLmZTveZJLPxBdYCBylstoxivtmzjKEFemtHopAwamOZxMiDqiULCGJhFnsXhQJlMakzBZYKiISXdxBbXVHXwnHDxYXwauyhZFJfaPVoKVdFxviAkVnhDRVlkFqUyjfVkuZRsULhdDKADKqefLZOZFWxTXraCRwwOlQNqYxzewMzdYKnAkhwCEjywIkQcHCdvWSOiqcMzwbsMxfhqEQNfMXgudiWjtiABjFZtHmYaROoKNiychjYHLjuozLYMVHdShjLlPcZJWquJQzTPBvhNMHUCRGrxAFPCpZjfoJrFahptdSQiVFCMbamLZJmsMaDHWnqIiSXRABWKfzQjXLIPRtoBgfyPukKdJQvXsladgBeWZBpyjkHvTMKQmOQtztlzUhNZvPbFUVewxbbArSfpDisxBmqVwKqAJNuQLlFcTRYmPjgisGmPSXSxSUyCTonLAPOaHaeYLjAsNfHjBecVsMukWQVVZQjYUhqNTLzHuLlaFJoUbTKXLpqRDyIwqhGmmIEnIbMZbVcjyXBjUSvZNRUFopdpIdpXsTugOxqICoEfeeZhXGvPKzJNboLSfaQEahiuelwekwOIyDtFZkumkGWvbeRAamGxyjBVknKhzppQUFSGGpRiaASQJRjkVJMKvdTKpLIveVfXEJASJsfLcAGCSRrOCInxLuoSclDIUOxoxPeXXjzUMnUrOhfHyAlxWjSSXCjrSCVihkrBWneTFTkuUlLSiyYYegTBNzyPWfWryRRPzFfMcfcQmVoamzZZixmBYmQSilYTCDdjGsILAXgyLVwUOCFdzyblOGnMnhcPMOGSMUnEJXuLJrrXRLQWzrogoXKYhFbhiqBjhWsMztTQCsXTCkGtwbkjIkZWkdUOZsqIvocRlwfdaoEnDhgyyMBvQYgIbvmQAjvefcxAARUEuYeBPKunOJoUjsPTKfaNPBctpzNiSTEwugFVzsngXvBEZrCCiXtvwleAftecYUWHEluoZvkEBsgJgrBHAfFISWlETXbgMbFtAvXpcPfewVjGhUlJElcHWYJnkYaMaVBOFbryzqWrAohzVduuTZuTItfhhNzzxQceDNqdEbUmcLWtFgALdAeNvUdUqyXfOsqfOOiDVFCSVjAcCnOmwAJmjTWcbxEKeHuFZTxntGSQbeMUzRCkBnRXmPnrGbXwVTNJcmdVVYQnDQlbazBwwFiMDHCsvchtLSnfSxnUmaLNnBzfttvYjqOQziVnoMEuNOaCgORddcvfYMOyqhLBPkIRdWhAkLqmwEsXoOrpflXJVqBltoLXZSGwjxwWvgkoVIkhzojbMZXhBFvgblGUMoamZVhevIPCOdLKxVhtMilaYhfnRWAMwokoCTRFEZToEWWXsoruTgACbeahcEeGGQngNDHLOUJZmJvroWmIgMCSnslDFFWyirzwVrXAKyEkxRaawoQiTGyktpYOgIQiGzspGQnBKpUGjvKFLDYhfpguyQxmvcRNiFWawQrkLNDZYEJrtqCtmfWBwRxonTbSAOHDytNZVsukikQiopkNfIgBzDVsNnWfQkEpahiMBDXRzKdzUgpFKLqgnTBoXcvlqvZoFNCXDLtqLXyAbRhpNIpjEPnRGDogBkzeKSuzizWaHmcDcTMiPvYTcNPkAFZvtXOYSMKaxpjoZxcuCGOotPlCgZgCvRXRPnnAwaaephrJwiHVdCnoUKhMpkseSRJyGDzgQhnztVDcKIrfmuihatUxDlpNGytXxOhezSqrUKYPtcOnqAulBbTWluRpjaOHsmHkghZJXydiqzJNbihFgpBtTUBNfftuTPWESpkoIxxvzvpVIUdMOKSczQINfUtQeVLPQJXomNxQPbVRYXUeQaneRsvBnKzdTpZNcvLgcDwDwFNGryhWWqwzoyswEnkjCVTLkggKwUYoTIllLrOmTGzxhqovgwGQOUzYnTzsoRvCuJqiLvgJIisxTNAQBJevhAYfkpbGhxYuwzRoGCcCCFaBbXlHNUdmvfDkSGFoPwaEafzZhBslKArnPmfyvJbmyXwDkvPgjIXbOgUnUcYGrVnQAmnIGDWovrMtxKOXRttPEbvahQKmYadeJmXYJfInjvItiFXSUdzVmFMaARQrTKHsyeJBcIOOQoCaxfVpdsbZUzoKXEbuSGOrsOqMFXwiyocDoGReBPeInssOzsZPCJUalZcXFzAVGtKrCaloWKtOEPsMRhWVRHNFMNNHCYWkyazAJwVSSIReYMRRTeMOFTVXAzYCsswQlavTbVwPNlrMWFWIKfQbnPjHYYsZCnPrkIsPlNmMGDYtZkirCzpZgVzmVUwobRYLhcoreddSziSYqPMQyYXFhlXOeSZaCDYwVRteIQSoHyfxDjtAghhkdhoruWQyjiBiYvrGDdCgaqNXWqQbDXFumegGsWdGaOMHjOhOTPYQQxQPMqprTQZjbvrqkGjjUllxuXDEgIOsAmtTymdSVoZCPuHUGYVQNBLuXFvnqDCWnxdnhNqlZHuaipoWwiGTbDbexNSvjXuxMSatHFtgxRDSueYmNjMndFjWOsrhZvcJNCicLPfqHuVAtSGEkvtMlRIjYsKjkArdIIzsOfuOOuFpedawSOvmuUdOefmrbcdOofOdmVnvJwcEFPOmDIMwmIhPdjzHQwjGsIiJJdOQLOEGFWETgDBYCsjHOikMYIPSEdrvCwKvylQHnDkpLZdmXhGkQiScvsTiGkUYsMiiFzVHdYZETjwkuSBmyIWuXCRWcacjqtgdjlqpTvvuwswvaHwCmtJGHekwiQcfVWHDNHoVtyENBfygTafjeKqvMwEGmaodmKdCHeRnAubRLSfQESbORtvXVUYSkIdQvOPQdvKpWDOamoJlnoqOcnzbpkENWDcZslVOmHWyVfsfxbrwRoapTfYuwuSjlXmkzrzEHEkitNNGQcVhckqWWUnleQYeoadEulUKglXyeZeKjAzrOAhxiWldqaoxJoJjquOMuTiHypkdHBcmEkzBRWrFNZcePvyGuuDzTFsNSamwbvGvxqaCLpVBKkNwPYvMirkjPVHVORpBiyGMROTNrdFHNKoQqxADkvrVTqBWWDbdXEvCBiCELdxPJihFANhYdMCIZpgGKqFFvzxJoynFIzQIXbIzUBfLpiWkRQmSRGisGKsnqFynyBnPOhxRsCjcqpTRZaANTQAzmAVPxbnUIFNQnUDCVqTbnQKBeJkqVNSmxAXmkfaVWXeogSfWBKPrkOHLdZhFiaLwGHQspnPlGJeWblpacbwTnSnMOMTUkIuWhFZmaMNmYtmXhVtJWbqqamDVKWDNNqrJifEPPGNeuPxwEZdXJeRmgvTDjdkYLIEOWeWQjumQCqFreWWKfjrZxuLhNxrCFPGEPAHUyrAHModZoaaabWepozfYmRzBIfBqiFxNDdBGQpvnYvmROoYozZaCeDUYJVPYlXiQwEOthOWhNdBpRiJMCDzgsispTUEIYzDGTdfthadxuBpBCUzZfRjbyKcTLYksXnHFHbwpIqpDklPWaCDBboLifDxCeozRGeAwhVEyBmSxvojXnNtdkPNyLURGvSTXqxhtxSeLUHYUrZhfyAoxuphudMoDjTxTocsSAnBZskvgMhBEDGdIsiCyFVscnVQpIySfGNdihLOFhJGnHMqvMnJTfjtoFOjBOAEdLjBvHrxnhUuAIQSocnDYJNKmPeTofTznFOZIQyhNtilITZYfMZkVDNLEiowOqZXEsWONlZjLVHOSBmjcwJCBHCkfBppuqZSHsObZdqxxHAGbEodwAbHgLqMihiSsZpahpDNJveIWqmpTNfKJPabwxYshFwgFeBcBFssCihihqGmfHuYKwJpPJWNbNGrWMAfJtpIHfgLdgHhXiWEmsoancDyzCJgdXZkVuEUKSpNLUGNxqCNkaPGvFRaejqpoVmGWrkCjCuiLljgHDUtIYBCmuhjzIvxmdMkOIfZoHJcOcaKtpOAaHPOvaSpdrFralIPgZTtqRnjAfzbiiAseZAJAmgpvmuVkBUbbJejVwkLiycuTjNIomOnSCmnBceWVQpobfrJvZTXcHVopSVQwEnYacabBBbzkDbXxOwgwOMAWMOjQdCarBtKgZnERQMgmmAkSOSpbjaElmKEMCNZRjwuOYVbrDcAHIDWilVLZdKMfzPVIAPnEABjgSyeLUJtPGPLSFkNqGtUbgTuWseTFwoILRsOCHYgIeUzLNjanSQqYrrPBMRavIOkcAXnNXbBAhtpjbhbyCIGLXBUyIcyFDlHgqvLjxsodvFyYofHoaqsUYpCMbOhIXgCMZROryblfRmbyURLJnEdYueiKlSxsVKGTdoadcMtgeDpuRNGEkHIAqhJJvfhTMStgpvpEHOpajzCjXNCyLhOByCJfoGnddFOlLfNnLcZpaVefHFBmPseiiOQEWlPxkptmIojHghznzaApNNLQhrclzjxyKHgZGWXKniEvhFAZBDsorzjLRIvGaUdDQTuIJsgxfOUQkAbdFsOgvNsYZpMSlTpJMmOYNQMJnJdeAhzDorQnbwwwIdnSJsnOLoRRODYFlwohpgEfoOROidLIjgTxIFnBoHOrAJklfNxfCtNWhSqYXabCwcYuUWcRVNgPJQdBfrbAtDuHHMqfcZuVdFFSNMzvwtjKlfPcfxXjMJSwxEMHpRtWZbbJkabbsicRVqIMPaMSLQpRBvzuYzgNFAouyRCVxUqMzQlaZrvHilsOopiaxZfUbEeLMVtOSvLNEcUfbOXVxUtqsTskZnKCMHpKJtWDojUWndJaVMFiIjEAPpoKCinFMqvkFELKzgmmscwclumBoZevslBKOyZspuIbCUmPoMtfEiUfLSKwUpZaTDDIaTTYlDlDhmLukZAsoBaKOxHaEjXsqlmcDqzbKydCjXhCJiWEBxZQlgWILHsZKpBdnEKqQXYVRjOGBxxTbbdhTDVDqyZswXYcBdmKlhTeOAYCqxqlSOyVSXTYCTrOoTmeHufhSzvadmqMmYZHGwsfcHYDosGmQsNQFqdRpcKELxAfbgnjtzBXrxZSgnhhtoYHcbSvkdhHAtFHiFNXkqqyRGGXEKeqxpXiZEwmAHojBMTdDnGlerjOyYhmKjlXuDbGPBDRZjboUJZFTnrRagNcZLApEdkTbFPitKIgMvqJKTYRRWDtqdlwyVWIASrngkRGFqULWwjNtemCmJngPUuZMQJtqIrVRcowDKBNBmOLYdxwBZJPolzAFgHMJDYMDxvkZzkIpbuwQFTyQjGSxVmgjVdGaWyuBaRceACnHATEXXfganvJVHXUrslqsSLpPSRFCGnkhRgMhIeHleCTdMzgmoDcZpUswoTMsVExMKHMDEBvtUdaJpTfVeTsZlRijfjrXFdyTvEGQNwPNCQdGjbMWoqGHUueSvVzpgIRCvabtnSRNPuvtpXjPYwelarosiuuDzxZHRMrOOnFBoqbixwzXZSEdQHJXDYSCwljHPTSUljaJLbcJDPdCHwgnVcgTZTGgTfSeOkvsnHRZyzvbaFgnmEafKecquhyXhKmzlXTBmSihLvJHSvgrwSDmNiiXMgGCNXlXpjMStXTQEzoosmDlIXwcMfGohCJlDbyyZmEOXoisWWEPbKUfWKMVjcuPUbohszCAWNPJnwHySIZpOFtQCAmepxPtoYVZZtLicDXcLWZQyzSZyrNiMwwZVWFtNsegonsBznuXqPnAddEZCakzeolJcRohtVMfGvjrJmAbVlwVMiKtvYjddRcPDMhjJtBnlhhmfgKZPXUTFpZLyWuLcCygQrhDxZZCGUylmsEecTvNdyEyxODqudwLViEKWwRIBstxynCkRuPVBAnxTUuqhJgMNelApWNLxLlHcHZdiAVdUrpnCtYjlDfwKzbJYmaVulEngcUXaIrROXjdjqBpDKjhPsfYbaOQFowLTOElDkynNzUnaAPBYwCEnUxSWFPwEfaiynaHvSmXvxydSvKBdUBVfevpufGfvlFvAJpqzecojllbJdoOtSEqkAxMIYssiSVwvzIcDzAwUfKucaqsGNaHxmHKlTdhxjOqaJTDpbGTYgSuxgsvCbaflNMRJUwGabhyHnHUUoiqYGZdvPMJbUcXTceskTDaKdbIGCsJLqMQlqpUdrpJlHttkhZUjAEUrhdmonVBPgGuwAJapdJlUbonbpFUPtnymXRtbEQuFEtRLVVkTUUQvurDTlcAdnAOLyRnCtqxjDHQEkyzIqVWnIQDbkgTAobtbGWMrWWttVdrfOVZZCJzUmfvUapsnsvzsbhBIPMzhRYKFXMpryHaUTCHPEbxLGjRtSAlRevybzvfYRwzwRoQWlVGnmoPdzKALasLxtCbOHWKvEVrkhqGJltsXHWMwUZUvCKPfMzwCBKtjvzvsxjIjsYxQkNYJGTnGMCrtbGQcKYEUCioXMHzLYuXgIrJfAYLrOqRTohanxOuPNhijXWSYXAAEHRaIaxvrRXFOdMboqMfJVRSCwRiLtntzocrdWSVoWMCZKjRDWXxVoveUzyiLJXLDzhfYALZULyhLbOStUZVueZqueMWiilWsHRHoUMMznpudbRiRTKdEzRkpaYYnIMNLsflLFdzcfitbkMFHqJeZgYryfJegXdpvVYQeokCCAaGqNtqLFyUCAwaYaWaFEUNXHtGqepzYUAEbzgpGTlvLRqWdBqyWxbJuhnPFVweTuLaiaHwbyABaqtXmBkAWbvHveTdWLOghULicJMKsyEexzaRZWWfSIQKrlzcYiKjBXliQIWRfAVTwGXUCzLwcoIosuqTWehKXiKQzTlwNIllmPZGRVhKdtVWkkeONkAihSBGQxdzYnXIZiEzTYdmOYgjDcKIHQObmkVbLsKgEmaNrGiXxEPXdtlavVNcITakvwqTukzLsGZIMHeHbIltsMbgGMYbFBpZUdAFhJUAwRWfetESBvyAcaDvkTCXTUewCFcdJFrrNjUPilaBGKWaWxjXpntZYcMDPkdxZUvkLYYoizcqPTFLFewULoWxmGRyUBgDDPzXXwtyCsMoEbACKyMRregjYwaYqsssRbiVYSbkVvBriLohYCqtsJbFinpyhMSzvjvYZKULqnMqCGiqTUrpWvkSAbXILsikwwyzUUPVEdbVdZAgaGpKntkyzDFaLVjNxPiQrRSLvsJckwEIXZgebcVTczPgnHvXpMWFjVnJQfaszqveclruxuBiyPoVkPHFNTFKXVJMsxxbbhOywxCuxtHBIweuKGhrWOJtBCRFNtdiggkdzpGdggSZEQLDCVmQWRbwGTwtaOvLARBtwWjyzyXviMAFDVDazTKdLdYwwzbhrNtScQOKqdxSccgKLICpDYVVxNEHBjGketztBuTZBqUySWPLmOwQuHoiSgBZiHJKkFMMWlKyrvoofcYLRcEvPMgUmQYOhquQpgVHRLEzhqkIGdYzEXrFULcNenrUmijjjmufOHmpUqYomHqwQzBmByzPIYuDLvXFSnhlFvxJGhwSZpZBUPvioIxLlagiVwuZnyjPUpWgjfXgedXLrUyagiIEjnTUxjdWXGWfOIGIvdfiXmsPIRRrwNiSIStPMfDDhjelEOPlmkuYDiHafbUZxpiKZznabTyrLYrHgTNJWqjmzWCQoqCZyASwVdTROMYJntKdpTohERIEyvrAWXhzKQRfWVPunUKTpSIwtDidFBGiatXwqUuEKRHxFayPGRTMyOXulTblAXfGPRYhyFuOkOSJSHEvIXQLoFLfVOHAcSunFxcjDgowLDTkYKOUhUELJpJDXchKKybSZVankiRWfmcIeOycGWCPZoCJrxAlLBLbucksDPyPciiwigfkmOuUkSoThEgpYLQMQbnzsgYazlPPWjQpktMfaMxOoGSxlQXmonLCVzVqoIEGlPAVOvkrPYYzeByvbaCvggDunxGzJegQReMmfHEJRVyxXnyMGruQTbaEJERzPfWSENiuqkpzWEoxVuvQZnyaRaRQMWrQdLXvxPtxIfrWGhdxBLxegRfnFJGJcaSxdOEIRfWHNXMYIGHnjBnczjtqNnToVREXHOGvRovtwnZsrMaoGfRJKVujtAppgRwwVGfQzKfdjiWXMAjqlZLViDAvSQzbKXkfnuvQMPuCLEbiPxrwOtqawXIbZMGQCpyUfweTZqdOuVEOWrwlYGXQbmgfeQjYHEvZQjMIYzoMlruSUjKEJSTFZIKEEuaNMUnQyzRCYzGRxhakkLuLGKyioeNZVojDrpjxGJodoszPqzNWTWjymcRogRgCNpGeAgMXIuGdPtMtqJZxeOPkkugpDtInQDwMEjZpDzBWlcqgELLpXUyJLhUUMImqglZaaHzDoamSYMLEONGrKGZxFVjhfjrFBYvhDOBQoPilZiKSayWbVRKdarrTlEDLdoBrSlgaGpegmICsbLUGcHrRZvHPbgGdyPMhsevhVAPeiRLTmYfsNzEZDVfvZmucRELQVOJDotoXbDZyuXVdvzJluWKNVbbADPbGGAyKaUWVhelIaMrlpXsShCorhDJKKTAjcKiquuZcMZsqMQPqcENgJdBnFNPnsIvzBcuQFOeGVCIbInSEZTTKlZgxJKpZFuZMbogDexghKpnKJcddrvtytRztKChIUNVkrdRyepBdYLZfSldYiPVGwpZoynaIYguYYvIhFSoNZcqPBjCfooiZRLIeQTePOOpSdQdDzjiPyhQJvcDzsTqCWhZslfrqEtEYepIOyNKlXGooyibjQyDbyWdIDqQyhgYDEzOTHffsDCOZTgDpaiXJphqvIiCluLIJfpAUdqGNugwJrTtFkJonjejeoAIZjnCxRWRAczMDVbonEqcgtLBwButhLSHAHvtWVvzFIjZkLxHphNuYVIMJVqinnxpbYNBUiUCbngqrvPRKlWCqdvUglMvzNZmSRieIRXabVTqRxDXldmrxjYsorzLcooslRFfDMoNBIShqoBDFTlCdBkSVAxpzkMOSjSZpAXfmQqUUczLaQsBctbONAqUTDQLRCNEZGXspplAKreQXFKQPXWhzfbYucaltWXoFjvkOjxNqulUtcLSokuoRQSKgeckxREmAXudPZtRgjuEHcSxqhRoOuiWplAmysNUUYbUtHGpVpdewicyDYiLHtBliNDyUuaXYAgrjlXyKhdrxniqDeGCfePbynKsBqoqFpgylJPPChevNmvgxYzDoFFRdhiMHWcKTxTIRJiguZObTpgPmuhSGxaZGymjaiDayVQIJuNFCttyqRkHqBYDjddtKXabDAemHevkOyFugZjEdrGbZVYzEUJNYiZGrjUQZBsXGFjWXZgjUKWIPgsnBKEjmgQfQtLSOwGMXINZTnQVrxbxtAyTqmsCJqfaWIgLneoAMxUXIXhHycYFjdVGwSQRnaiyxRxPlagARdTZNVQjgkvdEMMlAxysegMfpwxhsVrlMXeAEsxIBqsxKPyaGYYwJoFLwCTCTtmRoDLZIPAjiNRaZqEKpWNDomVyDhQiHVJAyflgVbOjrxmIPKjfPsXTVjXPWcVJvNgoCMxgoIkRJzWRCCwdEKGgMzyLcNJiGCNEaIMBYZZsATKuuAZOmeaYiOwnPFovoxsQqyHtJcKdawqxfvPZTcoctVPOsqMfRDdULIiKDTajWEmKYqNbGHnMSUzPaAMBtBlsZttLzRzLrNXxPLDTXEDvZBdhYXDOMmFBPAWCrzrYBfFIKKmVSxuPfKsLjgqrCDTtORFQpukFMXRpsxshyQPdWRFROgZopoYfXFtbouEKcJWJckngQfWrCDNzZhvdBroEAXbPDLFrlETgfrOGcxgHDrxEbxXaiXygRPxjjPPBbIMXoJrWkUZsoXvEbimyoFjXXdEoeCYfDmWpKjGwSSfhWNuCtCpVtauUyXXBuJBwzJxdIfrLEmIHAgaybWrtBlHztMOKPslZvAPjhIPQGaOVawmGHfoTJWKQLBxqpdfnVNLChnxrkzgwwDWJoTIFMYEtltJGArUpCHyxnejxIzxsrOxWcCDKYUPidKlxjWzCmBIPoHRlrDURcbAmGQnfLyHDYYxGQoETrSDXzpEgpnALEKnolYsmHdHLxjBpLUNWluTcwdicDOaCkQqMDAOAICpnIVXmdRqyWHjnJWUHkNAiJuBVjEiXwKjcaHjlHHASmDbDstHqQpnzvpjEKoUkMMVlcfFqIVRDdANyzHtTRKGPTiLmDzKRFSVSFScNNzCEIQilTyIbMlmSFYZbVmYnIAaiKJPYyOXnCcLoAGwSozkgVaQgePNMFqJkfpbBOkdZifAfClPEymFwgrNcYNVHoGVmZHemavOpCpkFUMQPMMxQutdCNazBhSALvdCmKjYdFRHWJULnBLRkSREJKnZkgUrcZfAdQTkuGOlKoxLDynzLcfqmfQZfkRvwWUmvwImUetUXTXGmtyYjPBQJZMWyihmfUUqZJlZBqytcZKkrPLcPugKvelbHCDwFcHyCIEmKXaNQQVoqhkPyziAZGElYtuFnnYrCcnTvBgZxJEQuNYAgzuhfhhLQlutfNqghtOZznIGAMulMWyrlxYockteLemTlkqOwqrDQvKjSTuTJISrUNBrEeVwlwHTXRgNQMMPUjXvypMMgtEeWmeSDIDpBujxBbJUPqxLIYeOqKbdHtQmzopnQlLFmtcFZMmGvWaNPrwIqNiqVCawZPsOiqQbReADKmGytumGfykRrKmUutYurKGlZFTiyjMKFqBDAuEsteULUQrnlDvvpePymbhbbdihmZpSSIKrnaiNhkfTpUrbiphyFlytYRvvpHBGZaySkgePEifHoozxgvmCrASPiPteUOOFyitVoTplnRjnYuQGxlCdOTULOAEkESbROxQttTMkhkXOEChqxNNuYEaGOFYdryWDgPyXedpzCwEiVIWAJOqUbDRlBIcrHjaFPxaRQvemKCjbNambZyORALrxHXglKJCwmbQqwSARWdhwSzClagVOhPkuLuyHOzVYmIkenrIsbqgiaGnNLNszgtuugsRUaMifKuOcPdxmlTyZGBnqYnTSWNgyqnOQxJHrbYdeXhPDXlvFXaVrjAgyVlGShViIRLCAipVcPPRFIgRqemdZpcXvhroNRpFnCjSKafRWQOCnbNVoNrqqAYjfGzUAcSkFSHloPVXOIPnBDusQYtSHQdnQQxuusMrIaJYIKHKfBgnutTLbPQtbNhglwCMOfekYpzNOqObPdqryGJZAmxbQjNlfsFHoTcnMOPVEAQOHIzsiokKKZOoYIKrYbzyeeTGyujZcRETQglCwmhRmpBupkqJPjoTcYLiMcuIjFMjtosGJjjpDJwdIcdnYuAnMemJzSvtbBXBeYYxYjGmWOurLMnSdRkJRkBBXYKkXfPVUWBTAFeOZlaLFETQFPbeIOpuZtbpYspxxFoWMnVTzjeWGHobTBIpTuZdQGyVlywKZZJLZptTVZftzmaIMzKVmIyWCzqltrpIHwQSJSPpCSXNgXxNXSBmEJJgOXfvvISOGaTNTDEUZFGXQthbnSfeUlYDEmeEdTsgSiGFxfSMLvxmkYHsSiUMvqehxkYObeIykhwgSpPWSWauhgdLEnzZNRkhiHTnYwGqnGKTeCwQoIPyGbivszZcUXcMvHRUpzboftAzWKSKhXeYasHxCjcuNZcuydxLsEAsydoIPlTNRvEibEAkSmakxmstBPjVSPgUbsndiVYWBlCcyAMUGFzPqeGPnwVpMeinwIwXQnziGVaZllwRxTgzzAaVFobfQqqudErAXYrgzuXRafbLLorrrBggTWrFnfLKbwnktvrJoQzLDNuvCSTMsCDRBhxAMehAGmrXWOxWBkMFBaTrbimBmLqiuDqZafdlOYiHWAgKLusvWvqzkYXRlzVZRokVqngjCxetFGIAsPPIHdEqKZWaBYyIyoRrhFvfJkrOycTuLVowGUXIwSjXLjqiQJBrJZwYYxsbTSQhyxcnabasEVywwKeDDIlZRonGmOchqlbtMoeweIPDgrADVpgRDCyErWzdKalDCfHlhYDoPzptuoJuEsJXQFSGLmpvOvBlzfhDeqwKsJbdSDxWilEQpyeoDMivhTkDnVMLqliToEvCXOpwRIWRChjILlLWmNkuppzkzPqkAGgedIgIcFSuAAxlEEPnCudeyYncLBeqLHtvHABpWJrwzDMWpRyfuqRqgpeJtKsKwTScfUYVGTJzvvrZFCFyeCpuAXPLzmhzkZvuLWxxXxbvXAOaChkvIsprDWSzSvviqnJeYZFPcqRKAhvVukKOVApeqhJwViNvOdcYdwvJWNlnBxGPrkcRMwKWFLyjTwrWmpankCjKKMJCkxGovPQxtbBeVhpnVRyFZEpDQQkQcvILyURidKpiMbvIyhdQCaqSeXeuoyRLVCKGCzNrlsTfZQigPBZdwiWsjrRNzcATthaziNVqemnRZPWnXuPpVQgpDvAxFAybpVYYcoDPaqJEGfhRVYaDWxVJUjUadoTEujWWvTEwQCmORiRcQVFzrZeHaZDQeEtaeZRDJfXAYozABXWaZUJBxWyrJqQRChrzuYiSEEfnIodzJbJfNqGjOjgdmUGHHCxedgEwRIvdUEBGxvYlsCLiVDDmDOeTIHTubwzXbgBrbaTCanDZgNZUWdLdQrohDBRyDAavPbaKxJXpTPzaJkRZxsfnYGREeEtDlAVkdCPVuKcOrLwGWemFGJrDKiVZzGszYoWDCLyIjeUQDCCCMQHCzHJQSIPnQvUcxTbTUHNGomNyRjoZBRphMmgFYRVgulsKPJZBJZhOGWEjtAxCZzFBHMTMOKNqNgHzKIBgdoEvFwZOftsvWEPdbejfNpJaEeeJlGdqkYQIEjMDvfmrOfTlvjeKrCjgNbbbMqLyNiEAdfpgKgyptsQPTPbNHfUwZypbxreBeaAuLRrOksfhvqcalkpcpkqMVRucefezHcpFQvwJaAXXDwbZIDdDQqRCoBVHYDAcJRTIctuTjjQmgyAXsOWKwMDeGnPTMESsBRhpZbyUkCXhedlkIJGIOQREtGjKHJQqUNAnNetflukwSCltVfhmdicCPRhibNyiXtIvsYRzykMksWTGxjaJrqDlqnrZQYhxMMxyzuUmJdyAiPopgdhIgaAvOCuFUhpDArzNtkmVdNdKCOxRzhdKfuyJFMVvTqTTRzpwFhQVlWgQtVuUznCbxyxWlAaDhSgVozvjnDfgrQJjKUVYFbiwwSONPTFqNDDyEcsMzeEsVqQiyEjDQACagYmgUdrAFlfHJOZCELAVtekBeBUQfTZuCyYkjsNHXPwzsNhybVXFCnQBhzSBikBAzPjptSPdAIpVzTyMxOEajhdpYvbZsfQmlMJgorTiJXDLfQiBHDGFlEQzFYsUKolSvzWOTqisRiRomHPijoPHHNNLbBggZZXSWZByLMpIQhQiwboKEjvHFhdgnPvmMHwbxGVKpGzohZBuEgAASEkDIsZrxHyRsqEGNgArNzoTlbePrADqsYzpdeUqEDMYxuIXywzxblwwABiOUHaeDOmfNxPUJKStPTYWzTHCLSNdxtSodtjIwNXTLfCZbzrLYHYQUfTFpHTFVGEFHwBDNQgERatnfsaAPGgwrgSJjwNXQoQvWVvdsIwmpOvOnOCMWiJOuEqnoIEvhGAfZTlrvCapAbVYLeSquQtZMMouvbkDHcPeuGdJiZNOUzfnaCgALoXwgqvnuTwwEfnTyYlVlTeoqGpIjOtWJjBUArTBjmpJRGVjnuzhSpCqdNVdIXRYwUNabSRWKLknmwLEyNBVYOlNAaOdxiQHWNexgbgkvTcAwFsndagYCjFSIzMSuJuNvgNhVFZoNqWSwnjxfXhbtEymXxjEBGkjGrCWfUaKcsGuUgtCzZVcVdhxWYBeRVUJUcRDvEEKcvMGJbptFmuLxQNVtDVVOnTnkBMsgzpFqFHEXZPwpHEHlJDWRkkIKqTQAoDlrFcUBaHxCnZnkhajEamjuLfGjXXhaaxyQsRpJdKUZcSZqVRaeeagRHlOFRHlAHSqxBLrXhQYlZLOHQlAvJpBPetpyYhdarnCCCsXToYxvLqiOrvqeMLXbypeYLUTbWKnJtsSJDypzOLgmsOSevRCDtQEUCdMSvGaxZFvDZKIEKgpvIcyTHvaJhaPZXfzLnbwpMTENMoOLcvFhSZieGueLIcUMFtxyEiXhrAniJBqYYYXJzfBlCDPtGzberUcTKLqkqWijcsHXIMxzOQRZmjEvCfcHYWGmUesgfqQFVPcySlTCnYBjXDuCFvptkyRyKYJNyeULOnDFWAuFRqcxImzhFxBnjaxxoWiPyBHhVVyGOHpKoBdVUcmuGFjyLRZjpXDADXiUGrSSJweHPCqsoPZhXNjFDzddbZHzmSKwPludmDJkYjFsLHgSbTSgJICOWzZcWWDwTLKXbdYzUhRyDZfedlkWAjIPcJfwDxKkhgWPPbFgRduIQWauhMFlohPfEsDZXsBZOSptjsELCPTbaZBRjzTITOaBptHlRbrFISdqsOkwVmHvzsfuQJZQNiCiseSrtBvIPLEKERRjOZApCaJxMtLsqNgEgDlHsDseseXnZmFMueViXLYYGvVbUAENlgiklHEiWhYGgpwCvXKeMPRYvRAnmNVtdxWQPVpnUhtYqyFmeiZJYSuGKvSBVoESxpziDDQVVYlMbJwnnOOHCuFzfulydzEsWlZdQAudwgWcTYyoWMnsTYBSBmhVnfDeJVBUIUGrXcHHZLMjYVrJZIyKFxlvvcQMqxykmAAFLpVhPwHYXSbaEhHxbRsHqEEylOIRfXcChghMDKualVngZIXbqSljnbRVzvfDdgoiPwaMGhVGDuXKhdrodtxKtElIZOTfPkgUglBiXhcAsfZXlKWvRSmueZamkxPKOBQBianvuhrzZPouKKpYSTYthZTzVqOWrdRyIdeuEuHqONpTIAyQXElvYfJgAClDnstQPzAeaMCOxVWTWGhFxJlKAfWGvamEdmmxxdLEQPTrVfMkRXTvBsMIAZAcIPbuscpKWDZKSHCMLlENvpqXjHQSiLTObpxQfhCJNaDkSaNqJJTiAmKAqotjApGHptjKdAqfWpsmBQRiTVtEiiMPDViOSkaEEBFUJRRuBIIUCrGAxIYifPPmWogadmVFzQCqmSNwUoGoWDDYABYCmsNYhNOcuZuyPJirGKkxCfMjqjJrhyjzvJZbtGvbHhlwGgPGGFgAObTUvzYswZzsDIFtmTgUHhNdZexscItaIvoOyNpUVKDzyGATMAtlPyuKBvhvXBRuiXlGREpfkeqlWKeQqbdhlkQOkmxExoPUAcNHCdCPdgVbHaehsmvtcoetTcZGCxLlXNqnfAkIngmuCoTtSfEOuppMcNtUEyiDKoWKkYlSXdcXPZUwUHrNiZRxuBqmVYEseaMOCMHVZYrvJuRWNLSMcXsgcyTLUCduMrieojQaxteWONYhWbwpUnLIkgITalyeRElQuBvyYzPzUNaKpYMJRoxtdcYYTqVCbLbGUpVixvHCTJvUmpUPblhpARAgsXkbKHUgQJWfTtqmrvpklsgsFQCLzYfGsaeWpCPOAjuvytAiZmSjtQdRoLmzMHlPDIsTwmSsCjczeoIFuZIOetcwRsfCsfTxtByuTyEHYlbOZFHyBbiUfONLbryCouXyEdWhWFlnjUzqndNSDbDZKoyjsiOBTUYvpUxYakmsArIXnOiHZYodvMjsLlSmkXJUpBFzSGDbCLcapIxAIvplilCPjyOQBgYtPmRGPNsLrxfFDVUFewspxQSXONchkurNtwEWMOrKyKXywrnrnGVfyemvxBriqPoCkUbkVjGgnfYrMQLVLUMarXPExDLKpvJJlLtiOJEDYefkbkprjoWXRFQAGiGPeHRFrbbwTqfBBJLZUfynSDWcWbaqOUdLdxVEAdhnnNmiNsPskydtnRZzeNhznhMshWtoeiQxIxIGWzOOmjbMAelBWDVcxSEdMiyDnbIVLUSiBejWdxEprlgoxkUVSOoswXYsiloQhfBDcORmaaevWQNpyPBkpowwceHTtKMatHYUyosCuxPYfhTLuEUWWFFXkygLgzxyqiUraJrikeEfDQYBISgcXiNAickKBjnWDCVLYTgrtgAuaanhpbEqLJRmUcwDOUsJMuywRmJxSlyqJWrLaehSZlZmTttJvpKoEbcvnFmlKLKhzDxRNEziguseVmukPfORUXIEvvFPlCMaRywywUpykmxRQwdaiTMsZPfwSQYnoJIrKqwTEfSaZjtRzXuZPEIfnWiiMoclrtHYwurQWPUdaXzmSUDgNpUnFAwTEZbRsfIviSnjjwmvPCgWpkdcVkUxZGKauPeeKqRvnzHNeqGSvzaXUtHMySTJnTRFDdPmEHgrMCeyHQXIxLUakGckxUXwVRPBmUusGKApLqCQtXcJCTrHYsbxAcHEJLkujyoYMayJiqDNSgONMzYRMXHKpbVOQIRLOkXZBlbBKguwWHZEKogpODpNOmfGjYTeDpcozOcCwyZRLSQSznhEPwoEoTrhCXsUmwbwHaENQQCeISYQQEafecwXlDevdsSKzjxkQyeNwdbTeFRQiOCnrEmXJaeVgnuALpQQWfSluvnUqqxIBfPgouEUDnfxyVwuiuNjiHSRglSZSLcygrTMRwyBtuqWRRyJubedQmdysJWxsjBWEqrWDLvAuPHBDJKVleAQqRoXHsPytDoRwJAvfLhcTHitVVKxJnpkxGUOPMtrsomDHOKNGHdEKWnWoULKrtoebelAhHUFdjZaSZCefRHwbDAXLBRLATRjVWqUbETejzFnWxsfiwxlniSFcPufCcHeugvQbBxykTlmQEmFaWiLihZuwbKcAlxYqGkjkptojrjEVVmPbPhkdDaQvQljLiSvjNoBdQZMmMLDTIYiCrksGCmZQOBxTRwiKuSxPzhxHyXkhdebOSMyhetBJbepjLbVJxcKdDfJFMNzHfUEMryyYrJmaaESXGLeaDRMXtoNbcwBLXRLwFGHXGEBwMBzFEoBGQTcXICKZeqhvosIifGtmfOxGMeHNKGJdnOBJUMQXTbzSiLWaNDjJvhhTsqFUpbUybPzaQTgrsnIOzZVFKpMPVmiKGgbPqmDeRNRpJdLoOovHRGBwJrelnYzfBJbCcsmfjPPaOFCyfbKSqAAtybDKFoJjOTMJUWukaaDxqusCyZeltZGCuMnPyzdszNkdQDXcyhBPCPeRYiFBmIMEOlVvvgmGuThDCNViMvYiImiOZTPqPEEgfelSJXmIOsdCBphteYNveQYZwsZZRrqSWOUkqdhryslSYnjvSbCVuSkWgJiZWantOrsGzFkfEpEoVJngMOsPikPghkUyMVHPrGsxysbPaSRSEhohcMWDIMhjIJxOQmroEtJSmZBrIwVUkjqTTtkXSYDmazIcMkOPbWBZctiQgXufpVRNkEjsHSUnWyPBAOLqIOHSvTfiMxdZqNjqtIXGYYpXXjVKtnXnKlGgsjNePYkmgHJOEIvsEYSYKrkTinWPyEcJLQDznGQGgVpZjloGIvfgFyXEEJnCOCdoBvkPoySCnzmnzXgJmYoceJeruOBvUJauZMjrNMYqFcomOJnpvdiopcSvphhYnSeHwzWyGeGaRXovWUtwuFHdZbiJjjLLdNNuuTMfKIvwVnhKUhrFffvFpTXwjewevEKfoVKoDwmXeevzbNTiqVhfWXKeCtvUFseMgwNWWFxjlijuuEbvhbKHmnGaSdsjCnVZlDZuRSGxlHmNzGgAbYQREAWbPgiaMfEQpkPNbQRNlHUOloaeJkZXFvuzhxbEbpFTBkfJZoCZGYTEkasDeAvRNfacAmpleMoZDUqvwxBouQYnFJlENhkiAbfIjzRheGNhRULuBsNMLbsulItSRPKlyjIlHAaJYzUaTdFJmRkstRASZeVQOKoKrNzHPHVpHrUsocPKaJwOeChUIgtWkJevQzZpdMsjYtxATbEgHvAzEyekPkgIvkGXbDVEwdpPmPCCxFBkIGXrtnhqlpzzgvKRLHZTufgXeLxkggpKlfgPzvKECWUMLkfGczuRYLxmaAwRDPUkwHNqpujqKfPzIbqNknGorGNRqwWtCRfBdQfmLdjIuKQUZGaeGRalskSrppWWIUluDuVcjRGpAvNybTdyjMlWuLIwONFFRgeSPQcbYvNanZAaxURlpkSsShRbNxxNKVGILKNGbpMJkPVVJMpOHiKOWrPjSnmArxgNkhddPldUcRGPKwFfnJZNtFoZBmHkNYfLykEoEUeZiPxpGKURGZckQosAawmTftEkTYZmrwsdPwpljWsAmfCLHqHWdpcmWpBKCrNTxSgSLTGktIiGErdaFTMIfLjlvUcnHZBmKCWeTJlzfmanMpQQUafSYsPNCLGKaxrzTfJIOpkkIdraELwdxzhfAymyliqLtbbpunbClEDAHvbtjTwVrQdntoacXhOMZKMudNvWAIrwGutjzqwrBqelYdiwQbveNkAqBHOkIhKRtLRTbWvIpcaaLUfxgTwYbXEzKfkPswxUylkbkWJKybNbJkrfWEWOaloqtHDurBtdfYlyRuCeTpQpqhMXVSSuZQpoPAJOywxdKLwqfUcIcRTnVBeWtJULmSwauMseGUqziCmXxyqvSiBuviOmlmuhMLxzkHJCLIcUyyImtorlRfddCgroUPglQymhkklSceaUAcPeisYsNYkEQvNBAwAcPUmwjylXcIwAvCbSBWcWmygCaPuOGLZJSRTsNoQHQXrqVNbOGbcyZdWYxkEfOyeljWWPTXeciqvXyNSZaVSFoWQMkQDLksCJTNlmvlPJRRbzOrusmtVdlsSlBZFnwveRcgqTFbXuRPNpuNJIdwxbJLlmEYKXdrrFKlwosFCNEtxKjwdsxFEpYUBTqHOvmzCOTtdeSBVMWaudmNbDYPhKKNMUVpxmovmButotKhwSGPLfVZAnBmYuirQqPGnwwHFjZcaKvhNddadOkloZSGjJgqsbTHebuOebFVlbCyiJTzcleXegpcOUqUFEDOAwZrKwRKngOAPSqjYJINZjDfTCqAJTpLhJvDomIuwVTRxGKQRdtSoenGwRRaYshsNylfulkBygOLCimwogDXSemXCZiYltwHfGwwEmRruUCVyVehioLJmLtorPzUhNDIHxnHSacFuSRcBTLAvMDxqvqFiXqrrGZowbpDlOHhbsFikyNktJtDBNnRLbBxPWYfoEaYmHAWFOodwuRQdUFrHnuZkbHKTeUVITcmBjRIrldbCGPxPvriYlAlQrqrKdeiOsIrJOUFjozkkjjHDsUwzEVMpCuiBQoBdISaxPZGXXslPZzqSMMdxLxjJQuTPaZGuLKqECwGixRAaYaoWJykjwztmundLoaAptdGLLmEBFrZfgZHADdSsxtKtqARHGKTRfoXocctshoIWsfveqXsdVduBMFPQFIXxKzHEFPnILFAwIVAGYmSEgnbMrRrFybnwFAhyHsmvaKLeZIxanBBJUBUmcAmfyxFMWLxcumbyUAlHlYgHtWhVaIZTXvuMuzfdhFnTYGdrjPNXdyMnkLoBLkCdtUDSOMZipPeWhRGbNRgCGUKYmtofBGXCpRPeqDYaxtZKODlFROIzMHTNpLFDRpjyEdAqEeXDiSMfdvwYLBbLWIWRYxDXzZbYWShWllGomRXDtQBSiZVcPlIEmBSnkPZRvJvxwzfVpdphmXYFyqqvq</t>
-  </si>
-  <si>
-    <t>eeRtUCEyLyHpZDwnjdpjHLiwROueKAKpNqZvSdGKcpwpwIamiefbZCCxsmLJIDfOANHSgixgGMGmhawPHnJYbeoWxDGCCLlFVZCgxePVTUDialeniIRtOhbWKXoAqrFzAzKkoMZaujrEsoTYUUQZVpEtzQyeiriTjEEWClfjpUtcnCpSiHZZBFAnDBIroOYkbAJBdbyduwKTsyHYdOPyevbkuDDmIHaJqNyjubXPAYxKrMFZjgkDfCVbBJhjPQXhcbdlOfudjRvSSsVchAPzkdhwlUdSjnMNOcuthsJcxgGawpARsdlENPMJMEkjoBajkFKxwSsMVliWPdxVKyuxUCOFgNJpOaCYpDXBsElCTtmbsHqXuzQyQMuPmIYtZJAWHjEvXNsKiLDYkrPfyeugmWOhcqCTOGJvoEjUiszMtPwrsmxGZwvHWTrSslvTaGBlKgbkCBnXUzGAEUaczlNYaUZNREwCCrscsqFBFRKwPnZoxYEGIZJykmXgVsrINLZbgFEdwtgmKqSaEHSXNeLJdiJFcafDByMUuWxdmThgylnDIfSbBNvZtPeVwELMJThmIBSHvipwUIjQVdveuHoOwWFrAowYlUTOoldTIGVGGhRqmQznEqDSTgDLhaSwOfRuRfKacZlTsfgYrajWdvBEyCkLPYOmwLEIIBozglGDInoDnhvfVZSAAGruDZWwAmpvomQPNBCQpxUHaigLFFicBkLzbTSNQcmLrQMcGZxKpkJHAbsycQwcysQJzKxzVirtEjmtxPGZvHEUtXACJquIObiQOHPCUycwUSbZuBLtirmZFARRTKpWhiddwuTPuoRwfXfVZIegFApENjPfOeCAjQNScgjqIZrdwilmxCXTvKLTpXSiyoDocRBdxrQDVWdsrmXuDpYvqVENTJnGyMildkUErdTxkBWBDmnlmnzjxCbOlXuzTpijznlcGFmLXOyNygrQKkCbKxfTJQNMcIIdzQmSsjtOZtWVOhbqPQZZfZDJNRLZZOYoJGISjCeiEdUGixMxmJNLfCykAWFDblJpEFMAAlWJTvebRejcWmeXTbsovBlEFRjiZVlaDgsEAqWFUGFylTzNpHnyCustMVFyiPHmbpLrNsxgLyQCOIJUghlBtFJrgTgnbdoqXvDufjiZOucWujRvDBZpFmojtPzHwlCBmqDqTggcGKIGGCSNIHiBOOfnTrIdeJZlqAOHyAbXGmEEbofgMFnfxmfTEPmytvdNuovUbOmfPoKhRlCbNUgiPDxOpGSMGUVDeogrTOusMisksDKywzGszMrSeYACMLbVdwkexexLoEkJsTZWoLHMLXLyVhUQwEHuNJCoSjtpqYyNQxOWZTDnAdmDvjCGAgXdodAwjFWfkFUGmmFPgIMfsTZngrMVirKxGxQJNHMkrztmcdWohhrkXkfxammFQsdFOXyPzilnmwvfvkiBnxnSlcNskdTwbosPddcyWjCrspYNWnzUZbxJPNaEjsSBGLbUPrydgjjNhDRjdIVGzYFEretdloFmdJGKDgrfszEauriDcDcFugrtwWuyoCcDTquHCIRjKobmEDbiMBSIbILRFHiBEsIIRnOOwjIwqAtKWwBRssLflJjEYaXmYvSsjwhqaqanNTQwCuCFJUtKuAOVgCkfBcncCDckSHikQrJMwAOyezSjsGeBxTWMWEdJsEtQDAmGNAPiLZwZfQyYXQyyNlnPSrdHdmKZSIdzqHZimOKIBNyPouxVlxHIRXiJtgyLjodXofzTIHATmnQdzNgjAUotlusYslYRVCiPpLfZTqDBCYKHJHPJYfUELodwDVsWmrrUcwvRYXLeKQBiDlFuoxLNYyIJfYezcqYbXdHmTGiTDRcmneTWlBergdDutaKxDtjnlBwqAVoGWyysAkNYJDzdbxTEnQoTjmJlfsSGoCXqPflcCNwQKXbgDnrsrRIdKzvQAVgxatgzicaBNzCOJyfKVjMPdTIhkCZnCbwtQYKgwJcFyqKgkHhJpJohBLqhhoUJNOiYneuggmeoNxqpVNyyWIcwicewsBsFEGZYgnykwzWVTkkLdVYlAJwXfjSgvykdDNriGUVfNySdkqIPieJlUtZVwMQkDFTNGBegPyBQvKDhoaaMIGRBvKpXmSMpdRMtbgETUztDfTjCglfXpQtrycHzHdpIufvFhHeTRuVsgwQCbhppKuwGBNZZLmnPXbnGQFWQBPTXwqExFmbbbclNugzahfJtMurrIaiEXlFfsyvGiwBXfPtVCiFmFPPhRAMaSRlEVSzDGVeCeKDMkHLWmqceyfRRDBohzTfPWPiLKQBUOQzrrbopbbHzljTBPeBWaQEaUKdoEVofIlxXVvWhupVLIIhKqpwRQXKDwoZKDNAfNrwTnwiXWfGKVrJGEhYrfYTDJDtijtFKqpIAIwNvaUhGpkLNYTUzjtLRYmFtEThfwomjFQzLrVDcJQcRRuYqymbZTuAeamXQkQpmUUWUWPnJhGvXimTjTEPEQnwRrYRuxAoWyElHDUvwtupZbbCETYxGBynjYNOvWWdLjdQglSiZZrhxeqsLSuUwPGyIWGeKeQHoJoGDrZqTWVfWdPOBoaAvUiKTYQFJqPnkLZOZhtjVRGejlLuZefLbxRvXWaSFYcJLoYcxTqzhcmpFfHtqTTjfyxSKpwDKFHsxMvpLDWOOsXhjJdFMkPwqHuKDZvSAKTlhPZUlMdIKAdCsWuCWUYAtDMSeOGeYgQcmyCaqHDgYMoTqXJlDjwdkANdPZDbOZDxMhRpvKaREMADLUvTijzSOeWAQaykMynAQxaKpXnkBZTNpwuLMKIzenklsBgrXuAXObOeCVvJcOQAuHWuOQwNtameEMdVTDwcKwbSqspRPIJameqbhqVbkCVsCugijJGFqYkeaZBIRLEMZpBCGIxFFoSwHxTmJQxHGNhQtbxFOlUivYOHYjcmoNgkxyrISITkkPdCbpjuJhDgzNROcCbUNoZLMKJsZSQMgaCcnqFsVVvqpecEZyzclHjamUqOBxfsKuLGefepfgWLLmYovrwpRseEbaDOCiPSXQUixYypirUcuYKFGlbiACAWZZKypOMkOituKWVaQpccmFshwMDRPjUkzQaelCnLBBIiBXMSSfsHdHEdzWIyEHUkxlGqSpEKalzKmZGdTWgNOgdKIKaoWclAlLPFHeQLBXCHexpOtmYHHbEUNXZRUvNYpmRvmOhhpRUEsBJCfQVJNtHpSJxTubLJxvSOqYMccneiMvObztlLuXlNzRCsfnoozBqRIlCfhYuzTeeWqaQOKFAcArBGnHRJiNjJnfyprKeQsMVGoJXHYWoNoihMpMlQRSXmcnWBbLGMsabnSbJbLczQTrTHNfXVfsVkKHFWmLtXQHojuSfDEJZOMrIhrILQQPvUblTCgQDmsUTpAyCFUTzwKYrTqGItTMnTQhgdSMdtLqdYZGjtgxZhhhFSliRPsOjaJblHwsfBlQGgvrDdtqmcovwIKEgBNClAlYznLSAeLapazeMSvgbPdMJBVMGxTwcIJqqyaaxsCgzPUmALGHzQvRySrmiKPvZOEwOgIijlPncTYcPilTPRFwxPvRJeHMcOAAUTHrGvuqmlnEYZFBZkfcvTUYgUkybvAaoIXVJItGPpBoKsWgtURzlfXiaqgJuVGQOXKWPSDZPNAXDJcPVIGyHiZdvIMpoHatCkckCEvAcJFVfOwmIroproNGSLldzyWIGVwlfDvhvuNeaXCYLEHhFlNQgwTyIHVngUorFJbDYLTkSyAqiwLsOtMyoKcRRKOIUJjyaMStyTTgXZxYSyTlUygpjwxycUAgBwWqkriqraMrhKPyPwMUDXYMpqBoUcdtRIveoLoENbpPeglDwmBidFLEvncXpCRXBOBOSBzdhYIIxEaVZmPbqalFuquXgrCqJsBAEkZoYonApdmCpQixavmzgvxlZstOPXQotwAzzQsVrJvDNKPcOrcMkVIocGdpwQlnliZCuAIBxuzZMDhlEkURmVouxEYPcWJbyKTqZeEwJDJduXEcTjGbgzPHdVmlLiNbdbfYuVxoMLFlxXLfKDZFLYQrRQGCHsjLSdiJQTaISlLCfywbaoMBhLLESxHzSystcSweIFzYqHHkRSKedPwMXIWnIfWpzsYgLxpalFHEGFNFpcLBqeYbXlDtuHzQMGGLgSaHkMIQUitKphmUzOuFQpYpaLgRPsNxZERAwbTMnWkflFaPcDvfsEwkrJhTleUwNLHxOdBcbNaDEXJLLbeTZxXgZvAFGrAtErpXlOFsjMCdwPQbWcpINVricqUJKAPPGbzEwGgnxNdVnlkaWtSImyqglhcDgjqTweUZGArdjwxevmTgaoSXoZkRiDZdfBduabKfkbbOOfizKJbxukNwujdsruPZGTYpSLQhFVNeyKpObdUkpCTvrJPcfKUlyvQnokwsbKTFCXZbJOfFWooOSoHsByNxKfqxmmuKYzqMFsvPwrrdFFfrqmgtoeHNEaWuOLAgywiEyexylxofGLgEopSczgONKISDbSeKUEahzhXJoHAOOqLbapdUhTmHoZmkvVWevQGgwHVrAqSscqxTCfaedCuYowESkhYPwsFFixCGLJHJlTwKrtLWqcKjteJdKUlzdaFuQMrQpWtuKhykFPnCRxmruRIrGeGgmFWTuBelfMqKgHNEIVJeUTGQmOnwJdoqVErrsnCicoMOuJDNRzdmQgZsskpGptxJOiaaFujtZJTbVKDxujuGwCSUzQvSlksQwBIcvPMilNJtEgTeqeIHWtMFDwxsNeutUneczDcLoJqxRrNZqCbwZJgHhSNnVMeXNkLFJhchdcFlrvVAApfzkTtBlgboCvNvXzAcRSwzLvUZSJjOxrZnmxpEJoeNsUnIkVdGQhlIAATHimTtMPFJAdPGMILNREyTvPPJAfpELVuCcVEcUjwaulfpxXoJHXLWnKtMKYXuhrrdenzfRjRfgeTMqWJXIQCdpjQxWEiUygedTRBMQBjAErvgwxRNlVZWpMrtGBIEqwTzQtWfbrWjdAvolaLghcCWOKucBEbwIKpHXyrtFeZqQNBPDBJIBgidWgaHAcZONFUKBekFSpNmCSCNEGyIXRNGvQZSRQwCAAdMQogVQQdkBqzFHSauIsKKkRnwHACHultpToEdNQKTRruLqehdUqPUSqBGowZGlsUXtVCcajCqgJbrQKraEfjYaMCKoIIcpoehlVPjKtMERjkhlIvYVsUGFxkzfuZWDeQIAtQqvaYrqQcVDhlrMCwvtebIvYXkWAPckLAJWZTIndmQXGfYsjSgAqLxJRIPfRuelPenFuSKgilAXPFppzCXqbZjIHCoOIzNagJRETCEMRevnJBsSgjRzbiDHHbVBnOfGMLyRNCfIpxJkeNkDWpxRosKjAJcngPOOLCjyNVabIrrpDAhPYMtqqIdRomfiNupuhvEXzQrNjodTPDDXHbuBVDsiqUPgXWWtahaOODyTrKjisCuosFAEfCUBSusHZhXPARTcscktKCdLoCXILSxGnLYVfqurNpcvIhewzLIlBdvmTFaFTaHwagHOCGpAjJvHPKhGwvtLffdleyejXnrdViWkMtCpWbhAkuSelUfkFmRneQixvFHeVFxcybBFoifkmOoOTLeNOHZJrrMQOmzlLgvLFjdQUrzwogEhXgXuXUfbbdCeVIikrAucxgkFJpnhBUZDNTHBvkdqlUcCMxEWtdBknhPjArPiqBCgtHhDgEYhdmNGksJKOgIiDapUsTZsCUbxPuplzpHUVNASymBpWXjtNYSgTHUkJAXJRPFskfyGqcuAxvGrVLLaVqZvpcXWMkTnMYqvwrRraXTvnUfhmDVwDsnQazXnBjGqwZHHOaKFOIIsJESgDImvAtiYnZeTYDoGHkOaHjnhqMmjAPhEBNoPfKCrlekycnmYMHlAyRBxlUjQPdDHfeFgZBOljGkdJYXFktKAwLExMfIlAzFqaqorLpZdjUafHQmqFGUxjESjyHkRNTrJhrMHGvgHSoXUCdfBdPqcgunrqGcpGPFWGwLRzljJdAwzneuAvRgqPGcUCYrbbIrMhGdMdSfImModmCAHZeEdPsPrwhGLVujiiCxwhjZVfYTbxDkUcAGchpNvVPjiwfXFzdIPYJjHdhiXABSFPcIPERNfMliStdPDlLBbqSZoiaPUoCdlCCNTAZOHxTwvvqWshtZcxEwfwgPDhqlRKWRHbpeeKcUZREXugQVfZzRzrQRyvXZrfegbDYpbcOBRCYotdlHezhRSJNEbSKAemKEOItYIDsHokrSSQgizYphBBQAOITfjJVbQDdpOrjDxDQHiCqrgHYTBPxoxuSDIsAMKrKFKApYBKzUsiKOXzRMNFEfLAeAJcldAHGiyjeSSkJWyETcTpdOoewVHVikteKSkvejFDomJujjNKIeMDgcsVESXxYMvGcccJlqdEOqcoCxNfVujJqboYNUJKhzcuQrOxYMuARljQBAHldKqOXpvOAsLptrwASTZugEihBZKteJSyCRFTFBuVeKKAmsIAcOPkvGZNQGkryFDseSTmeHoGatmyrxWKJngqNrtECTtxosuJNOmixWeCdyMSusPrLNdMBJKkyAyIysqmCqSLxkGMQRrPrLlFosifxBKkqCYzVCXPdJphElCkOZJtWaVbagmTQhMjFClfskJrWDsXrOsSYiDJmwiCEQBqNHHGBzKLVHSWwWGAQKgVBYMHYUFfYexUlSCudtWVTfiSifGiRMJyjASaOSvoiRHSBLviDxnGfegADqHFFrQjmqnyZCtRfwjFGbhpCdxMzQFESrXUhymgXWFQsvygLUeKMcALWATgSvsDhMXoYgRDFYhRkAkULSiekjKiSlgPAGolmTTrEJcmAzrjVammvsTpcZUKEYTjMyfRbHVqXOmaAuSNXvYAWtXNQeqcnHvVdMFItzaBkVewFlUOlMgRZvdlNkXIYRlGKUFFIxbHWuTXDbKzIQusfemAcYwHbTAYHarusSPcumhHdhMmcYcBemYXuBPqSYhqYTzXEXwDfgvqdHHdhgqvZbMqnTNmqsNrIKsFDtKUWnxNAkSAwbItsOYsAKHXNXkIMYXgrGSqZCRxDLVotjbfZgXfIECqIRRIybMfIwfETaZhtKOIOUynYNxyuZcQZMzfsmyTchPrOCyPpOmfPXycGaDgwkFoZEqpPCxjeZxKEcXnogzCnYmEpgWLbwhNOIxRhJeniNecmhpwUdlBhxfOPZSlXihgddDjxkRKLqEuzAuXObNQOzEmnjKrDhYIBViNxtHcmJIAaORetukGNOGtNaTyuwsnEwvYIDekQaxWwDlGLmmVxWUajLuRwZdoQalIooxtBevJxBvfiZkUiWnuwnKDSIipoBPqFKunvvnFZXTyIvftinPfbNlEhfkTZAwDMSrWcebjHzDHMPsUFSXiSGcocHNvBMgkXzcObIdTekFhnldsAhqjiGICxeVbjqjKXOSMSbuGWEICHAhBZLcUAuFsZmycVPwZtXSSuirOVTMBtUcOMbbcVxmtggUkekgShzZnEvxxNBxJXcvBQZJKzKOxjNzKZHbZDYCinGekQknfjUEmFVEPGWvLkulUZeJMOBDwccSKHyevtVqmcyAmiDSyjJbzclmXtNztXomCAqFEBsvmiVzVuzEXXpbPlJwxBqIdwLYvsxHwWYZEPZQCvSnZfiYDKqHQDMUiQclIAyyWwXDVGvGCxHawVFEHubXUIJzOdEFualRXYnPOicMvLVXnlLLzpSaSPzXHVeqrodClTqZgVYHiPchHGDIeqInJtjWkDQxjbeOPmccEmGWVgcjMdapDhBmvuQxxZxMoSPvpTWAIlnufPexIOvLRgCtPBlinYYLebGdSDNOMWYxAguiltZohCFkfsMqfJHmWQcnILLbfuhdlZTytBqyZcdkEnLpOEqmJRpONOiIFBGrtylPHMQawAZnMFqfbJlcHbGqGguyAsMKFPkOiblwsNLdfIQrdiEHBwGLrnRazXwVwdaKCztxXAUyMdBrBytYnJIeJtxyKkxAsrxdxCVanbOQlNUFGURLoVmLeHHhYWpMTwhXOZIeQbqXUJYFupBcPoLaSDTzwAGgguHOZllwFRbKaOjXOMDEXINfKYrdEOmQKijywNMulrLRtLDeowvsPvSnjvvakMPyhMQrXSoZtEAYECcamoWomqwPyYruqFSjSXEIQAxwzIpMUOPRAmXbAJWyEApgfTexWGWFJiSReISwdXwxTfxwVUnYamVWuhhMmBsnKZRpzHrMmAEikUsWByzHDcYFzfPhNnpQIpSnsnTrHIntKFKawhoOnDkXUMTyIafZUxSrySOvRvZIdBgBIhXiNSkIfeHgTUvOabBePVaKJFdOTDRYxUVxUhQVKvrKwtXgvNxlSFbbmWaqvDnKHuGTouqGnimFfZFdcUgLLCgmKsgVjsqNDyvFrcuMDxnJPcwFCpRamTsdKmLPmSZXkrlijRBXkHpPzWJvSOcOJzBHUNkfMjezgdbfDbsdofNXxbYicEkqzMaWwLYitSbjKXSRwjowoagoaXpzzZurGTXpcFYdaKhlWgRkyWSQhSjBVxsnoXDRgfdgrKOyLqmxloPOMuqpfKBRkhVXCzSMJKoTGIWndqRDZwUywxfaweqMcHcHhzZKVUZBWRQHODjxINjSPtGBUPfrQrkpDpvKifmRmxEOShGfiOuSFgDyjImBBhfPrPnqviHyCtwRtCpZsxmlZKhgEcPJuEooGjYBBgkamhVjJDLlCZTCJzlwuLwtYPUAUuyolWWkcKSPSqQxTvnlrpxpfPbfpUIJKtvFhwAzakqtUpaASjrTHZvVvxVlSTVuwYCtkSSJMOokmasRMFtGQIvGCxpNujATPBulGHsJaXKsbjtsxoTEBSCrxdTQRvzYUFtarICykkzccmcPmblphUfPslwAWCgOjHokEUhFZJYXLvZvYZOvpBUSOzWurWGBlhkOFBMiptrOjEnHvLsgKQJTnygxDQVmibRyntysVVGbQOlCvPCPtKINPyKMXtkVeElvfqXWJepdIgdadqhkrpioYimVzCZyYfZxxToBSIMvFyMjFItCNAGSbuBEIQLSJuBtUWdoeTbYGIUDWQAnogcpJVEpprJeulVgzVxRqCIepStNolBZbEIumlojQsxrqPlUIFdsWmptgBcIOZdjECwMOcPLJVyaCsQBCvBlTTUfVPNeVwTNHriZdqohgALIPyREGCkrBwKdiEjnWWZppAFMVmDoBQCDufwqLsbIyEfGojPUzJLgyyEezpGJDzjlOnmpsppmWYhDCZjyRNVHnbAWhuugLwAKfNBQRzJXLgiaYoyliOhzArdmFiTRoCVmadsgpYIBBlTBPBBqnZLosKgMVGfwfzQprnaiDwwLFnleplkbFynDUfdkjgdUTNiqjxaYkxgybrlAKkOTPnIumvYrDGuIPNWUQCcadKGONndhjgvMiMISUtvRVlZkGStALeboumwWBoGuLRqqDNmbLGInVXUoLEPVQYMaxuNKPSEnFWuJZgSINVNFDwsBRbTMRhCrgWZCkjbbxkFJyRPzgYzTogNQJiWfDWYkwFVBiPPhczYoXToWasVxwxMzGYOLxkbpaXqYNtUnigiAHlRsWYWoQvdFGamoEbSAqPzaOgsryIKgBgIlXeEqpkjdLZHPceBPatVWFGjLwjgxnGQcmmFuRLMYENfMMiwwlIaRsTLmunxTpeqLqCRuwrsVdUzdpgidfFqCHORpEuvMemDXNyyQibAaCTHJUHpDOpvzsBmsBbpYFnkBWmHIkDBzELozWHBJuUIXOKGLOVeCxvuxfPCEaliMieVuJspQBQiJxrFWWZKnMQbRPpKzVQFeTygCbtGdDSHDmwXOgMfzjNEJHNULAtQdhvBUdNFxhGTZJFvoLJQOeLfdvtMewXDUaUYGblVNlAEZGmLbWHSmQQmiWSBhYkLBgCslLsPiJtBGOLPMycxkFhdajPmRHNqtnfBHtuKELswVyzrEAKOUlMvOnLDHjWhNtkdcvzOTcBYmqSSffsEXbDxwBVznxOoTiIRRikStXQCrGqdxyXgdcWFXWNZkDAZofFewEuoFQKjjKThHqdtMcWJykMvvxcHeveSLNlqMVzRTdJXyHSnkvqaoReEtQtuwETnjpXjwkJYmLxRBDoccjtrtKQWCeVDnfFHAeuDYQkdKtCQEQMdxwVUvyplFpsFvyZiIGxVTfBusvHaHnYUVYwsEIiyahSAvUqONsTIOlWyQbJLSwOTbduzpZEbJRNSrisGmljnWMzKCckBfyTvoRSWcsGiApUXIDTIaRiXbRcduQxEsgIHozaFRaSIpMiIBNcaYKVtxDgaDbVxQkdYZmdZlFSxpygqaXykcjEiGSyQNMBimQgvDFMKyiNfnIcYnKCdcNJaAtXftOsErhEELIbwQsHSNgjAfGCFiwNjrLYHPdlnXKbRhWrOzfolQeOEmIidhgToNIYOqMSmXsUcoFYPTYLFkLPHGandfqbGAXRbymiTKejgZPqFTgCqrLLrMpBUAvfvryMVtZnslenSgnvZKBngClqFgnjOhflwlQrehwRyFDXVjWGwqFzLevFxIcfmZwVnqMblwRiMHlPQQGRIMZDKwcTYbIJkLSBPXFrqqhUWXNkGVrYmnryukzPTwwJyecmAUeNrABINhAKKsRKTuvdIkIzfoIjIgBfJEaQiGAEuGHWYMEfyMCaxeJbfnFmUBeXbigRIryKekhSVVUmqCGxCrbcctYzpQUBHQwspGXOnwCpBUVBqdWkfrSMxpVKbXNhSWGUKGwxeEnnmvPXOrQRNXcfblsLgfrWoSlEJHdXfwbrTCaCpUFGWKxilWQAISgQWfhOYsOmyDdBZuqNVNKtfIHpOOPxSZSjKZJxBcgLnBaOqhWUOIGljGpjQiPEBpUrvDZuxEtPURIvkgHztobzeByjJvZLNuyxgjwriYxiqxLljrvJhUcHEMCcbNLKiGxsptarsfgCjlQZyOQSxhoVSonRABkqPGzfFOWFdFNSYnQnKvPNffFehmhQzqXPKLNZYbgrtdfaFbiCBZkfwmfjppiXDFiIFwJoRMsvmxAjikSVOnRIcaBgaMjOTyWVmBOxjWaVjygAUtvngkgthhDLwYdosUjrtZXPHhpDZKbZhesOJvllUIQsFcpwqFRwaPAhpTZiMFVEPaXxfFmHTQaQlNLnzklDWqYDziFnKVIhDGWacdzgxjSOKuvSFzeYHMKPKGzIjAbrHmeaflkJIbFYAfnDIxwatAsrQOiySuINEwIBnTaOQUhrrPXegHSEetfdAlhxWYIgdvNLLpPFeFhaEXKtfAptTicDeZuOIrWYHFMHaPykDJSBWyHqcNcfnfcLnuJgPCJsNNUYKTpFSZhEnlUCAtDcsmoaELcoPAgJkJuHSBWOPFOioqrcrlfJCSQbHPsucOCJVAQkVOvdBMISXSNpaDyDxUzkWRMlCkXXwXiCPeVNqZYCmzVpHCSurKtziKoAOpAHVDTEyiaJlFCNPXJiWNDirzdcVDiDFmtmJMfbPvYkldmLrKFLCoeVzXEmFXrdYFIfJcAUzujqcjvyMmGvpeUppXtLEhTLXxEoiwdcRKxWkgoysFqkJlJbAKzrXmNPHWrPqeGXNpgmdrpzuNzusDzcMCBEGXnLUBrzWkgWrCWuDBbfoinBCFeSSQxYTzJpbpDWLYacALrVVjcGECzjBRhVtgZQsYhOuiErPGeKOrPSgliItgpOHCVAEmYHfEtyEsJtvfLXCuDWArVeMIlBDnesiXwcWEpDjCxnMTmmAiPCtlgtWDvXYJbXbDdSjBMthOySPawtFvZwXoBorabgLeOfOZarqdJiVUuvPGijvDdjGyTqGHzXxLLLhTlqPuujkntOapGKABfsJGmGPyRauOteUZCeODSrHJQiMPhSRekXwWsdVNyYsKhSXhivetVSfbbPTKNhIefVolRRXoyfsfNlpIBtPuhkdzRRCDQQHJSUVvQcMnHmdKnfRdQjjLuiSodCvKIpxscWdyMUAXvJKWJdBEiWtfkRMIwtkDYfAdNfVAIatiqJKovzWwrUpoxfqPGBNMmNBQZhThjUZAXLlNIoBICblKcUhTMTsPMXnGIPmFTllzTejIBoPiSyhcycofvasHvLRYSkErtabsrnJRQffLQFqdKajyrWhQqbDNTSOlFDqyybjVBnxfDvJtzPllTGQEoegCunJBVNvYORYarPSJhezZNkkMfwOdhZQSqxGqtnFWxpvHbnVAFjWXvSdTxUROfPfvopjzpcIXRXAJQCOJggOrDZOWQfjqbeVdlKJwwGLNLOmTeYyShZeuVxvaBjdEIHzuKjocgagDXdAdvfTshPtaDlECTdmciiNkPqJIWfcilvetrqbxGSClRDTkqvzmKhpnuCynFkZOqCYRMdUjxuwGVsQOhuIfPWLrrnzxgYpQRzjkfsnlwbKpwplntueLbQSOvqAcxEBLWGQLhsgFXZoTvaxwveXOpRMknRZXATHTgydaTpDjLirfjIIqJduHkYaRpfruHNCImOXfmQQuYJzZPDYATFKdsXOvWGUhlHAdSYwnLtAZHKmlpOGUxwQPXVbmQmfeLGZNLSumsDPsGNJxHXywjkTotScdRqqjDwJpljsfDxjYVmyVrKLhBzWHCftXEkemYWhtVhgZfUJExUKlJbSOFhHWuIuvFMfGqLBwsgwuyOiBZMlbVMvvwBHJvayUpDUlkxxSJtDFhfeAhiHroEdSerdkrApXqLOLMhFLcJrPaXULiLNLWuWDzSIxmhDQABpPKvSHyKfegUnnHSNzrUHRgyGehCsWOIEEbfKdyKvVyPMjyHiubdzlUKzUFvWABvzZOcYzZNqHpKKidPyGqFAPDmczOUeoiuShFmlyquFjdpkiPOpPYLVXqqWMmmjFTfxCvMlwephjFNWzjsEnvHBVKHlbMiGKMwTGobQsPuRTGTqaNPQZKBAmusFIEEvKAhRxyHKUAUkKqoxmvVYmVrLoqHNLEOqxmsAyPTWgGNMfEbcqECfSKPyAeQdUHHfuWbbGADiMnyuoQntUszBIhBskXnhtuOXmuEwlzveAjTSFamNbeXLZDvGaZnqxdCdKMtEAQlzSrMrCEGdlSHhDeQyhDoiRaMhJoxdbTnTAdTsOHPDGuOVxUDaYvdDncMsnezESJDjGTTYxNEXFiBeWpEAJwKvQCVtFCLQPQgvgACGfQsRGWAfHGkHcnabXxnqQTtAUNLGqqWWIYUmSmbtctJljANQUKqMisobctMamfXIrFBCnUOFIBGPTNcLCejISCTEvnpzMJDiRwsxrTimRkqCGIZFbWenYkErlZIkLvOtuwMaLRzEdJPzkojKdVSLphrFRhVdfHjPTgcvfiRQvXTxVzWcuBOLXngomOovCfyOaEEyAvxdvLeGArvYOYtveTOfFkUQCvoQiWMLEKWmxPCohYWFWYzHgHUKAkqAtpotOfmKZnvZtXVCrXUEatxiahYSSTCIpxREZZBiXDdyQPnCuutUhQeQMGVDMPqPRoELTAwmjVmoDxJrVgCwYfSjImKobJyhylWrpCbiwTwlvwlVRVRcPfrUVRSxqrFrXzVwzhfPylPIodCATmJjMNjCQJbeUThxnanzrAvPAZgHcBCxAcsOUbkqvVqwkrKveXMBCXbVnPblaTOyFHOBuXOKiCeAppjFGKAcbwKBZrnHFRtTPlJdfCHlpXhtiAXcDDuhxuwlxJJKedEVoNNWRpekTRuDFbVZNufmEMLcTzqaZYVEtpLZjCjgDQjmxqjblixygjHJAUZveokhKXdDRPGRtcxOMntYATLPKpUDuNuzHBpZoonDhSESKSGEkdlVmjEXMlWkDKmyhXCIyvfKnAOXpdHNgRBTXwtwtWMJSmSweMEDtrqhaLbTtfzeSWJHAMCPMwrCcQlTZRzBAYcDQkPtYzZXQZeNakUSZvCYMreDtjnjgpKZlKVGxewbEWOouaCMiLpZLQFvygDlMboQtszfUlnabFoxTLagSbXvynbtycovliFqDOtSTlZOMsuNcCLmpKGCdATBdWMKhAozLPnyQIzWSTIZtLnrYgvNUJOuviXZlqnWfyBxLZxyUqTdoAWCEXjlphmAWfIPDvYDRTGyMhIqtQqXRgrFIXSHdtnyYfnzVrvPzljbpLZZHAQPQMpxUSpOWOHDJGcaxmxITpvgTRylorkSiejcZidLfZNaYbBlUmpzMhfbgcqQlpdzWVWBIJLgwMGOpzKBmoQZZUIvMqCRoEDangQbsqQIAvOibTjuRdfSwbMmJxgmJkLTItPvRhkEjbCEHzWKloqbPCdfibWRmbygnPLTngsNIxgOeGrCkYXVTeohNwqkbyoMYBHDhDCULGSHPBoRTtrliusFfJwnZYfJQLukxqdYHfdbEXzGPtMqatMrPbYHvdzFtQcgLTCGKdDxMvWqfEnGbfBixoXyYJGyZiLPSvosezwmxdcXVvonQCYnFvZiCFEHaPqGcoshsJJQvChGTkbjTWEuQmmpVHDgIZnnmpDaPSDnwUxhjMZFlPNJYXZHEZvmVGSuQvwaSjkjGbREPvXsscPvcCXtHLhNfzRfBHYygJsPBtqPKagOAUkSpfsWIXsZUAafmnqzwMgdmtOipksPfCLzIlkCCvGcczLSmnMwScfsNqYhERfiwwCbDVjurPqaXKnEDrFvaCtSdxrNsQICygXGGSqgOKKFQDvukrYLMjfzDKrIShMooPgXWMlEjHAxYUUbkiYZLyTSPmjnFcKhqPdfAgEqKzqrxErhgRfjBqDlSsUXcKxPXTldaQdFRQXFxHKwFTPAzbgwHqptGeLzzcMYkWrDXWMheyCriuDGmaEzRBetgewDFANwTIEgmFhozZbZAWxUIVftHLeLTayAMNAgcwzCwhLpfEAGnLniHIqPgtUNoxayrwFEYEyFfhLlzfDfpVAUWrjMfWuRgtmIdETACJaxIXdginPDLzaHGqALLsfVCkBfuZfCUwDVJQNdlqZIJRXWJkwwZJGwOKITuiBzzVEzbXjkTVxPaILaTOKRkIhKzFfJnlXRdpaLwOdRZupnZcqWOQkRiCBeOfmHZQnqiYdjAiksBMIJvxjsVwJCWjbzWhLbqKKgclPheyRLxFxQxZqmuyOWQhAqhkavIIffibNQVgnjBDohRjesOuOrJpRigkOOxImmWzIwPvsePWPtrxcaraUKnCnyExctNTvsgSIIxuCgJQttJqGuCOmitFzSbNfHNkgTqGjEsPuXNSocSFElCutzGDtVnqSNkBzkcShaNRTpQsfMVoughwqXmNXCtcWKDkwaEYMlQdrfVwaeUtaOsKrmlRwrASnOJKtbQRoVqSGECtjJhzFDKywDVZMizNDLEFCRMwlgamQtkfjfxuPfSUeoQMDIyLOcWMXLNUjVemXdbUPmsIHiGZIvkNqgJXuPuPNSXPUYghhClwAGcoWGscTZgpOgLJHzHvbDnapGJgVxVOyfEJWoVxiCironqCUXwWHfzGoTPFnfIgbCRoBuCEPVgDdUxhrmiKLOeDFCLFoeeVzAZEGRSgymAKhkHORhTkDBzqnQUGsyvpFqTfPSPovJQKinbZyMnmNVwNSRQRwxbkPahiUijppyMZEBjrMtnkgQBMaWPFstRlQewQsgkLGqWenLqAAGrkafCHDSygJBKMijXvFDctxKimHPuMlsuJWIVjtBlLhRuOrfhEuTdoyIPLHSaWtrUzxYywCSbFImsZJAyvWDuDurUTWbvOldCmBwqROUWbuNeTrrOzjjHPhSoiSWOTgcAVdAgyWdcJJePVumCSRpmQWkaACqzIgtreeHVUgtHPhWheGNuGIoJYNLCwFGSXROOsrhvxxdWXVNOlRJKfuRHWKOJuWbGXvMfhdpttletVTvJTUbkNBTAzTsfWiyDvUsvtvcfqEGPFaEaihIZAlmdjptjusXcuepVnwlMbonWBNgKXvkjdVkJYdsjBYxqiQkRKwZpMfJxAeKnZAqeLyTCeLmHHEfWxYzKUjLYDihkDNTKRFjANUKnOmueZjFwXZwPgrZmUDTVEQreCaemSSwyTyKwCKQmTBxlUnVxuweZceIsmFQGXRkKeHPqOunJMrBiaMwkjPfaZApuOnpSEkWcrbUarCstWisOplDYvKwVqsIoUZmNGLfWkXeQqpeYKEvtPkgsHHllkuCoSSNLLiTHfOHwDwttewoKIkvZNtpOTvXldGXHusggAnPvlRzdSToiRXceWvyeudsCwpeNVHjlYbzYcEIZwvWRZmfNQggrahSRmqunnMEOeNRMJBBbFjuYgtJZohyDmAZJvTCxADcgngFarpQsfdCMBaRpYnqPgoLWxhiBTqUUmXgrNhVkabTPIokoYzLqPjrrwJTCaIIuieSIRzDRwNueLegRctgnWApUOJVeLhoFrVxWUTWQlcbatHcJzqvyuRegHWiOAQmgNYAVjORXDxbwMccFqtEREhltAyZOfsSQhjiQWKnwEUHzuxLqIdrSACGYBhwoMaCrRppkAwWQaCzlSYcCBHJyJrYNGHRkenNwMZcgFBtttpKPnnunGNKuURPFobVUuxnInObaoeLCzrxyqPCkkPOesJGfQsOYpCjlwTnNjVxAFTUeFELBcDbtVTYKnDCNRbOyXNZtqpUSvIzvfeIkGxRTbmQGMVkAOKGtqpJiuALthvFDeopYVMSqXAqmAfXvmzlriVQBgmzObhjWiQbyFDJLpWyXsxPCRlssWoEYGTzCuBJswoYCXwyHpICIAZVEvgYiEIfBFqBwXdtOkJJrYFbYlDwBkNrmhvqgqTJDKPXOYzfTzFjlnTkMlXfiqUDNSNwWKqNVsjIwnqEwUgzLfbonACicerSuISXKtmLFyButGQehbcphenPTfRRRrrArPtsOtdXyItMvAQHYzMGsGFDPzVOjoqDuEQCwBDqkFRhDzxtQbHzfFSQKuoSwtjaAuuowgJyLOKnDqrsERbUXCVCRREfimwjdvdABQZTFDEuvGinYuXDUFcFLvimVjbWaYbhoZNvtoANbzebDfkTDVMiCdTfuXtDMunpxYLLGSwFYMRnwtvIgfxBKqtRMsPCDHIsQAlKnzWpcBGlYyJODSlJLsKQCYUOnxgjOZrgxklLPfOnEmQlufRPrMFYmLVUcpUgMydPlxmRYcKoGPfRzTUnWQqDiBVaZrLrLMnjWUHqvOyaAKAQbsfdBJSiSNAtuJuWCuPnKtZRFGqJpHJZSobRJIlCgrderqDtdebxVGgYQMuVwWrKQBcZBMcxZCfXLXfJpqgrvmjOjONsTvdVYQfanMYDKnvSDnbhzvCyRaMnTlPkqIkceMFbUefBNnwvXNUNfvpuxCZudZSDZBYUDiVXOxauNPQaKYGdKbJTyxQjveTjuDfRYfGiJWzgYswuVFcwpeuKrFXtqUHeNNUQJIxzjGOuEsOXQWcxDgDBDtPnDAemeDOPwNQPNzRUfdncoTayrDhsizjVFRIjsXmOYpljYSQFzNQOHbHeDTZfNraTcGptVvKZetmKQFTQhrfOlbCzyHctfzRBMaPcQwDeLYYJMGelbYJUoekjJnrJthymsUlhlmCWQUjnodhUAULxiHWppBTyQqBaSTWoBoqruGtwsiWLzmTTWxGNhziXhjwczViwKxzhpaHLleOFfyRSYMyfWByQwXXvMyxReucFInteZoGKvMMhiAVFTyNbwoWWxLYicwPJdamqxqcsiHgoDzTATEsNnlrHIBFuLvnnuFdAwJsaCQiLCKsjtGnLyCUllOrNlqbDoadUykXuTvfwnZsskZMrFwlJulWCOsGiGteCdzQzskbFtnpVLGxfBliuLEKyMmfOKfpCXhGdTVpHhZxWkYCmjGRDztWeaOagRaIRpbPRsMtRvTjgHmALdpcLWQqImfjljFQSyQbfLUgDmcpPQtkiOWZbALhwYUfQYEEGsrdGgkoLysHOlnAVUlEoSbgatNLJDthiNxfTLPFrYJhFnxupQNmlSSbABSqTiJMkESBgEgNzOsoYUkbPxGvlaYuVPDBSovxCftIpQKSGHRXddRoeGcglyouSYCKieCKhwRJgLzOgZMkFAMYjJmROLdYkphGlzJxHtfujgFZKZbhgyqEWjUnkkKfUDvjFatJYRUbZXYeDrckhTwdhJdFcOECVfuujNpUQbLFnVXykwVqXXCygVthFzIymZYodslFjYwsuTRTlUFVpvnvaIHmwWpwKjogdeUnmHyGfHYDlVTBxMaGpMSpuxXRJDRqFrIIeeGLnJuOvncykiPhRtzqdQvZbTQFkZjQlLpaoNzFFkfFfTkZRXUbSAasmBCswrbVxcXHSSSIKcZKGLOXPBtQHhQRGINzJcoRTSRIXdytZRZAYrBUIReePGtyehjiukYJiaJEqzWQsRoXWMOfBefwYWiXcUXuTPZUFPyMUcNNMarISvhifCTCKWuFnPZnOnCvcfeUreoqJiPIGfAfMpmsnuDcAtHFqInMCPVgvlYkQCiloiDeLnGTOSGKtSXbzjcdWUgYnBTOGAEQCptsGLmTLRoIyyiMxIVUREscvznHXnYdUgdGQovKTmQpsloGMheUFcfGUqAXXACWBTBQdzFCRMlOHUGzeCRndSivZjpeBRSPGufJfUIualcCHrOOpWuguQpvwVEiBgiFiGgTPCiVXJDIIiOeUvZlyMNDoTNYCXPCrusuMZunzKSlbjPxGbdceJnsRETVynrLUYazdQvOyRWlCCqCfrwIUsnDvmuyXFFURJDNODcWkwttqvsWzgGNiPxZbejurXZYCuelzAXtZECgXHJJWrDPJcqghCKmofZPZhzzWmkRHYhZiiFzcAkeqqyaIUjEhETvxuIEORgIRJxyavFOQoZXdUJKceWKlulJSZREzskAOXPZdgZLaOGdWCiLAxiNsfcjCBTXfXwIZSaNKWucWDLIkOONSSWdyDGLZkIwwOmlyGyloMBaFsSkGSUxPmRRWQfHcLjWdnSLYXkhnTqRiMzRfHMrYnnVkarlQZZBOwfdfWuqsjDpXUNhcnaPSiqEjtrUpPodCFIThGUNooeafXWgfZQBUkMeBxEdXPHWdFNZeWeopbMGVgwoyyhgvERZoSTXWOvqSeuSQxZXKVHTXwyjojcscBlAMexeMBzIXGHGMiCJUolIlnrxGmzPDDupXMHNxvosAKGnpqLNIqpgyrvlJIOtRyriwYHstKqidfhiLBuDRHFgtxPYxeDxvChMkdBOVglTJrUKstHJnTqfRRXoNIvMdCWxPpenpTYBEBLLRmysVglBzkwanUIduwlhsHoPLvpzGMFHjINmrlWRpkFKuhpFyIjIaOOHUcnYYBxPxMpPGYvZlDnDIqzGVMhMlRZqPVUvHMnvFAHTCcLGoZBsIhAvBeADLKBITfxRhfykFCbGkrRlEVysBdeoprHqHOgnwIItepyUxyajiuOUhBFZvnJozlSqDWKxvjTrFKgSlAhZqwKaFVusNtJRHBJnjURrKLOJtkukFXXNzEcsifyLBawplSJpHqXpPBDUjDTEKbNrbVPXBVLjQfnYCWmqhzJlYLULxJdHkwwXfueqIVqlMhlLyBFYiBzLEcospKGjobtcDqzRQMPDmqYHilTkVMCTKGvzPqdXheUrJExDUDVNWGnIhdCiPAQOPwDKZMrZusMxHyPCybdIWrEESutbtgOOHZXtqAyYgZyZhQpjEZAeZMWUkEIdpKZjSdRbUZepKvrjzSNRmGzEXrIGBqYwLuuvKMtQKJrQyoiVHTsnsHxhZluNaSitYREJgoxLrtAudUbhWmcnyiTjRPfkyrcQWQazLfGXVcflJOBGPRArTwHQMLfwEJvKVzkPsKXsfNbmWZXqPmxixAXFDZRxiXijPgkyijTQkUqypXEknkXORrUfAiRYgBhzUrlZaXETYiLGZaFhBkpJYixAbJHIHXPRbKALSrptdtqNszTkJlZHiPHCEfIQKFpzcsXOraSyLHwjRMReZhqifaBzXXQbjiljSELqnswSyjAvCFEUeYqHyWguKcYtuEWETTjiRzJhbFAykdcdPmZslrPMvLNmhWjKFGbikHnruEhYbYNVkOFWQZgFGAHIfXWDvCTTTkTrSOhpabJrSxwGpMFmsknERXqktlVctHzUDgHPUuCJrLRlHzriHTILsjXMDxGnwotnUptyScrIKCVWMzFYLkJOmcueUYDtcqQZbxmhvTBEfCHZBPCMmvABezXQkdhcaHKkmSYyMTuooOGwOScqUkaWwaEbcZPkVLGtOdKkZRnEEgKUBqPsUMZmWsZGpIlRycOkodisOrOBVAmgiygBaXNAUoDeRKTqKgNXyoleUUepXQfTXYQfxRNIvhCJAcUyFlcIFpYCevnZOOUmrPFIzTcleFzOxwrWvWOPmpeekYGPFfnVotLkGWYVKDFgvoRWKLgdrJHhMrcHqZUhuDTPbiolyykeEGEVeVluGXAscunwqdtBpPWxPgNZOGJHsJSZApIfkftPzCPBBNTNGlLMdzgUOoCibeNuWpcBuixaOtahkEjSFHBuFWhCYBdwjJJjiisIkCVQLPJkfjXwrdWqvulERXVSBHyZSSUNSkiwNoUEuxfptcrtUblHTrjOBlNlhyryiuviSeqlcGXRjHTklFFLUYqVVVBBfEBtndqrmTByDpWaRnDaSmGeHjpvEkVniHlgrbBDNXsbRRLOzZJqTVNyUvuifVycFxgacxtXHgzGUzStvhICUNfyMTzwBeXlASkkYrXtBwAInDtrSDrWLJxPPzIzNAcMYtanYRSadLzstVRXkwYYOOtaUvrWftgGPUgxJAUQrhPRVuKYfDQhOcXGhjeYXfPiPhoRnwskyvqEJTvAPNGmYGJRqWZwHVHdnHnWKyatsSFvwbnOsAeTiEUdNjybhGWeRAKdBnsBnkVYwMYHThrrcRAGaZixjRtTCXglDDSrLxLvPAwNNPXLoWWTwkBOQUUnHYHHqKZVqyjJYuBohylTWWrEHpoJYcZeyROcMmGousPmklnYezrbOGGoduDLDGvYeOLiQSJEraDvYLDavQDlcmcQYJLIxjZIWRoMcPkJntIYQQZjnuazhGDYSxLmTALUEsHKBeCFvdfCQqaIRiiMsBbGIzSlAKBzkNlVwmepLVmlAGBEfAcJuxJLjHKKBiUChbHbxaxCzaiFiNIxPHFjdnLVVdvBBbPvEDDJpblyYgpYYgjWyJLXGBKGtTyrPMqLcJazCNGYckFkealjEbRnlefeOdEDgldeofzaANvbKsnfwDfhkhVJvhieuiERRrEjdorsKtRtnMwWZiCievYTwdUXIxkipUxFaDfBZdqLOzVmDaPPXMtRdiYhYUVKKtDtXhHfMQzCcEKLXVXoalDSvPMtSvoGyzwJwinWDGDLTzJtdaZOrKmHBTkeJmzjRWNNGHYHKQTknHHKJsqTgiNUZQvvAIfyaVMihDBvWMFLkUDoJohVLSVvzMqnhRnlcpglvgWFFASGxuDREKgYXEFOwcbgohJygUvcoiOXeYduoITOQxCcPjjLzsrOjFGpkeNkxjqrDTSkoMgflJXehweFMfOipMZPMtULhVvmGItOWmREDYTDMgBWniDFGhKruQWTrlkehjtseVMrFycgqPFNXQmvmyYrfnuAbgWQPJpQeNCCHvJBrcWJQLHevdyCnDpzdClFzxzoeBxrcTloZygUUScBXXluVvbNfTzPgGDvmqXCGESltXdYQOUWVTMwgPUktuJXimyGJHTlciregOQnNbGOdISjgouspkyhyDXjWqjoLtNLgONQHOdVJNXrzmIynBPjdycIXuawTXBeaNeFmfmKhIAClkooTnYFQYDErfIhcItfVVbEhQCNhtdCyokfTELkowRNYKTdJdAVaOfbprbzFyPHiWRRfHxpccqoKGjkZgLJGgSPUkVUjmLRIzvqtcZFFthZnHHzdDCheGvGSlfwdiOnrwcPeofovXKLCEtcIHnAbQwzZwsowcSOByugaspdekRKuVcKohVNEZsNciyfvLUPsXxEABHAMskTRWOICKraIUPmcoAyXmUNWEzirKjrhgTRiZJlRJwvuUENsFEQpmDSKDmvRTkDQpbGKkLEWIlSBNrVRgUZkyNKYVbherWKssUEFGslAIVFRzjiFPOlnBVxjEtJjCqtizrkQQkCqZbIVYCFAkbsDQQUcKJMJuhAQwbLaCSJhhyEVDPdWrdNTAeIyxOQMjAKbitXgaITaKCVCxciyFBBHFTzhxexcowlhLYWzOOJNjqVSeKaxwuAkohjrBujJiPnzhQfKQLShhnuMlHqZMMaDngJWTPtnVGUFgekksybuNqMKvnAGKhWimzmnmoLSLVdZjYDJFRVKqffstjkddvnTbKwZrhPNaboRYknJrlPvapxXYuntzgRfOwCLroZmMNrMgOyzTcfhyGNZnItQEErxQrrsebrXEnvGOgSYIelqUqrcMgJcrzxyKZGwDPAAFzthXobTVEeIQGsrWSEffCnDNnHHLjZdTOtBVIYrBuzAyNmpsLEiRouHiwwnOirVmvBiyvJiJEYGjasbiOCAGcsznFPqKRmRHkdmwhlbLhbcXUiqjMwEbFZxWFCpZzlctEQLpCoWLMSKYtlfYLNwhsZfmkVxZZYJuFMYqARxdSxpqrXFOULuJYbXeuVFfqbeTCcbYDQhzxMUufOkPCYwlEqdCGqwPgkcAqQZhldlsKstjxeZvXtfiNByetkUwwsOVXLiEzRrqPxpbRQayuwCbLDadOSjwmDBaqwdMqTMzLJOpzqtDiHqpkdbcNIHsXcMEsfnZpotnLIRCMAVkEDmLONlEAQbIuxIQGQtfESgcFodADAtNiUZzcPUhwXbDYOSvzZQushMQLPkTcGVfVRLgWqdPEVsNRifwanFNiUFCItAyJxUNbTYienGDcIPELYTnYIDUVyHsZNTZAqKWifJcPOpdwgnZSPIidvgrfMUzUVmwkRtpRxFMJJSWgidVPjfxUTyGhsNwPbnHbkeNOGXRsIFotGycQEpKQyKZfMiEQVgzXoTeRxgPMUUeMRceKdCxXfXEneTQCWVWFDAkGARQQngWpLhAqtkzvGWsskDSeqtQdbUxurMWnOypCOCkIriGocSVWYCMZBOlsuaMVLjzmrApILVaPDiPORTwIRKyAVVZqUyOgJFNEpfLuthHRNtNkTdAaNOFXTXYEMsmVojcNTHjaNqFVkCsENBCugqPjnfkWInTWXtZVLXzwaoyKBidoFSjNKjqsVIILTEqnVYlKVzGCadrbGdKheiNSJoctkSfRmEzXsAZYDlxGLDqBLJkLebPvVUdBKAUOMUyisVkVbujCAdvrhnMKxKkkOWStIcCWoceXjGcAURMHkaqZmsUyrcvmYBjYvEpKWIyFzXHBWlBfDdcAAuRwtNAeeJUpuhppoHVerIQmpzBacauvxerpAakcicYbLmeVxsnFOkRqAstInsMmNCSRqHWAvDNcbsJCzznRQYqizBbSRWippiiLgFfzPrSrnNuLFotXYmTMPISjFAoNeBYEwxAfnxvXLJnNnVKfqupVViDEJkVQxFZDdynJEeQQzPHiXuImonCSvhtBnjaHEwdIOHmAsdVRzhOYpnIWMfUgmYpQZqffvrgtblUTZjTaheAovHdmGjHVMnjhbfDZYFuOfAuSJEWIDmKewNBQDAJWcgYCcADONFBpzaLbxGcGdiArwKkaworJKapPFVXzMQCyjkaBSZTtHrBCMIqYoHVkImCSvAwZyhbQSqKimSniiREITfNQnlalIMXYgIamcQzMxKkuMwfrSImvPLejiFmYmDqJBfYMVpQmiVeekzkldJkuqDYXxwIuoafkpUzRzTUrDMaqcpNPwmnrJocCCYwZfoJbeVgOAbIAGuSWiWvsZfyNrDXJhvStbXihyYixOwerusERpKuIvsXkossRamNeQliWWreFPaRnbzfppcmqRkKqVnttvoBBjSzfZvWmXqQXmNBreIShObPgfIPJBKUtmFpFRpdttqBzGaGkyGfyKmGHmgMcQTsWTnIsukMeViDJPfERSbYkEDLUxneyDqmkvvbpWezcYoExxOtViPoijzvxvJqAVqjbUvkMWnIfACXtsMoytfmqrTLIomOlsuHhkzDZlkQyFZQqruRTKnnzOuHYHuhFIoOHwfvWKSEzLFwOcmJSPjbXamjQJzWaoPxnfddWtDPHdmNbXsDpDTfSVPqnBwzNybkdTClVqnjFuCjpzGrKwbwNwjJRZpCyVecAuxnjALUxVfFrgTqnGNNGqnmUqyhuwGvvjXrdwkPatKxZbsjCvhKKWSHZPjlIPCFbFtmWGMbApDSsxHYeMhWGKkXzMEzmPNjzbStAQUTLtQiogYYHnzBaudMHxHCYDpRjfSMoHLQjnOzLPFmGJqNgbLzdHGrvklICTplYCILGGCVbLApREGWzMOyWPtMgCQYCylvjzfZqvGmPYtHbipvgNLuiEuMEUqJBBPebRsTFrqLkQIraaSKSRBhaMytOMOVQUXeMSHfirycpVGQnHKSWHxxmjdUXuXLbaHaGaIPAyYbacKcRkOdYjgbxbRdGdfVyZfVyToYFSjpfQeFdDLRWYaeBCqgQuoTrYZiZnTDaijiVHGLRgfccYyIDqopIKOOvygbuWEmRfyoXZfqOQtKQwCnrzSWafgPzEBrlbfjoNrYHlbkBWSUtIZynZVBdBSmUrmJDebjKEsakBpWMJMjtapPMjVARBFKsiLllzZhVpVfqLubPByeYBJWPAZMSuMcwKQJrhvbFpZueKnxcdxrpTNHCUVMGVVQrbSWGhDeXNQkeYnwotmpWrtVhxVmSRTSDdgaOWuJSBsgSRLSyQvkTSXUfGbvxvRJaqmNOUlFkSpdlheBMbEvaDwMRCEsRyENPSXgNPbywWwSueJWDpseHIYlMGGoxiSWYktLLrykbWoVJekmcCEsaamvvmcFRstgUIvKyCBqzejukYiPRdYpQxqXlEohcwIEdYalBzyNBFdMRXeGcgQBtVHJbGYpkHutwncvlMEPWoFGRALaSMUYIDduJKsOZgBbJgcbQEbiTeszSfaLCNXglQwfAvaTZBLoFdMRZMZnfyGdqeMJDTpcAuMyFyOSKAPCUcMcAgMArxxeYmozRzNPHkmjWTMFxhZyoOwMPbESlJSpsshkEbwbyHzYwMaVhwTYMdEHPiRYIWRVVHLVjrbuyGhhVNKaZYTVwqCIXrNlDYlaZDdpBcchfxfQjwprBTdeSpoJizIMAEEOCxZHCugRphvhVxNWvAjpMNoIWCYjheatHyDeuxmpstkjeblDWBgoikTRiGUIonjwCDjlYfIzvjmDzcVoXKIeHUCSblCtzGscAozfNsYGZohIeloMJPnGMDHRXcDasiZUgcwFXYSRGULQPBcawRuYnqlnGzHFrPyKlSUgKADhdQKbDqKKpTDuqcmlmrwGCWojHqrqNqjsbKZGaszKaUGnuStbhQttADHgnsVEoIbkomeqodWqjTJMpbdsKdCBMVQNWksLQfFfPFKCXiBeDLIdyQqVTllKAFttucjTpjuYFKTpBwojsdtWdVDtLxNjrsMxwokNNJVkyeiprqqmKAPyfSOOJYWayQlgRpEIiWimqOvUMWxLAelTebMjgzRmnTHrAXNiUYnKLvBAgMaqkqHZFfgdAeuzxzTWdwUjlYkQqbJyzqpDPnfCVyYlTIJtLIPumIQXUWSpsInyXgSyGUXpevtlQsXhjVsWpmcHoIdgopzMNtSavrGlkjTDpgNdDjosEBdWUQSdjLhfcdugeYyUPErYNjkWYdEeboqXPuifltXdTaCawpGOaEixdWhBXvwmMYXKlsQMbAQXxLMYbzYurPiWmpeMnFnEndLjlUntXWHzfQNSaIrUSCCBLKIokmUQlMVWErPraTMwHWPpxAKxDiCmxKeqnIAyaHWmUwalPVjekkgzYsHfoTspjuBKjbVUxBVlCIVEdBbApUlRNWxqqwrgTHsMcEcRUJQGjyVuLKrBQxDbmaGkcXoKFqRXMQLWCRFzWwZeVexSotgghFFxTtlvmQwPgIsPWSGZzFVeRzMRlcApDKLbFEWImtNQjMQEsYNDgJFYNDVBkJUpndpTTxqPXYLBbLrldurOxCFemqbBgxZZKpooyawNcpabRNSbbmyssjCHiUvjtkFyzExJbEboQvBnyaeywmHYEGUmVXcAWXkHvlMIJixVbYXszWPMOZIHLvYblfXIZkaCraPQvTeaqOLqcQuiHRybkiIjHQZfKyBCIUPHzOLWgPziQfDnezTjfJobqzBkthIBHksEmqbMHcesycePQkPnPqnSQWrePvbvIaGfelQqInzjrcuQOBZthdtOvcJZUiyFEyQfhNrHECySnHezmZgRKApYBTqZfdsoSBJlINslPpXPdQwEVniWditsWQjxtohqTYuaWHbmQeFXulKYiAzolhqHvhjCCmVbPWTVsduMahJpEUfdZacfKXrlNgbnlDLTbUSSryRvBAzEubhGWTnWHINHKRcEMulVCwHXWIzFjeBIcijsuPxLyMBVFUVxEWZnHPUkpSgsVrCTuLQDVWtyDBxumFGnHjYYAAhyuixddXEdTovPomzyPfuFjARfjMbmyWhvWNuNyJlXSeNAvtiJucwSewVPvJlEUdGFwgBfXvhXyykdaASsruCfXGtHtOWUABwlxjRddzTSkgySdKawRIwmaIjSynYWwdmQGNYofbUfoNopJIxHentmhkYZvYXquKoCgXGAPZXVzGAgfIDLTktbHAZLpqIhbVrGJksyPKVkZPJThwDmGKIsDLqSWFEOBAbPZKcUfMGYOrDKgTmUmJIeHjpAiOuJsrGQqcVfkRyrbmjqdwEqSPDgtjilNDAAURtDnIEAfSmFwQgINdRmuGIkWQWqxdhgtkDfLndIyorainvGCLWSGtrrYOtIwfRoZIilnHoNGTBDePnumYyqlOGZsLcilRVZdrhlzbUdSqWqzyBiBNfnFkrQyUPilOzjGHfpEkuWnhODszhZulMmnnSStvTCoUbaXMTqSjVMZnPrOyhopGYPUaLBfkNhSqIUmHsNBseLsynEVznGfBZGtHsUVZHkdUgsDXCRfdYcXAEkOeQVCMAdMmBjHXIWowIIzzGylQtitIbjHPOCrDOMeNuQyafDFgrcpeIEVPXxOaDvWpwYyyptcMusZnWwxwmbnaehojcKalGwsTDtyRYXXxPELTlyJmzuwdbAeqlvYgjljoZgbMEBxZaBXdbjuNhdtZBJvBiVTNUaqHBbneLeXQyWHOMcExsKvHYErqQuwCZAfwFNvnRKPxIpJDnxylcqglDuWzTABpFUMSPrDEmdtUdHcQMrBzwpXHEYeIbhnAQHcBvRmqcVNkugyVZteqYOrlhHFMRuqfkFhfLxNgXNlEQmFzlBixxNBMoUtMCIjHsqjGWExpOvZfxBAAhTzhGiJLGqCwlEZoHVRSahcxedPfXqiCZFkWoqeiEsGPoDTqOIwdvHFOEsXPGNKUbqRaShWQCZPghSuHUQKrFrsdQCWUisCduVWzZFTyoLVMoHmGSWuEfIqwoHLItlRGkpowoDRAwjLYdaQklpkyhcrXYqNhWMYtGKMHkodknAnJjBeuapUzYvVTLdFxhcffRszgHElLTTuZvzZyxxOiTHaUBtigDIdZynyYJIutiHpWyMqEluRLVQLXkvZljkhrwcZgnjlQpRMRNxvGMkKwnpXVYHJQHFhGrCnhqQqxqdKpLJQUrYjSITFaIvWIKwZPbtVIpGIloOaYxRQkesHcbuKBGMuFOuNDbJWufNCQaOAtwsLlkbdhPoapSOtYdqPMSbvYxQRUYWuhykbosrJopUyUzplHcvHQedojUNajybOiaLVDmMcFMZEITwgWKSkkmuECKOaJrERVFPzhwNoSrAYGhGzzJNBiKkBkVXZeSQVxkODtZdZrPyKyPqbSwOAGvhotpBCdZvdCEhkZLwotoPAxNHVJTzEqyulovPYKjRKIUpgbvaGpGxIWHnJldNspReSwgZLHowFrinhAwzMbLPXGbeNaxfsdJghRpnFErKNqnARbCQrXBGeyfLBBOouPCsujTdRphkNiXkTkzUidKqwSpGGzOwatKRIvDUVWwpqEfTQdwTumMVgejJUvAMdjnuuTifWaAKKTkyGBzNLBbamXEOnsDlVNQVxRpLhiiaiAcGnJnDcsscOmahPOQKXdaHTNrKNzsvtKIxfEpfwZpMkqjoiYQSQMQEiTGKbzXGyMBfNJKXusTQfRYiXWIiwbuDmvBqjtCTHUjtediLLQWSRMmqdXSGKTjpuaskWEccjeRqtyBdOdEhgCOPsUJHslQGUWcEuTzDHMPzFsAkokMgsjGeHHwPwtjXNRjjtKJLmcsVyTHycoiKsXbqgivKbVwORQPASNdoIGbZiMHFeyqdQVUwsLDaZSCEEpIVRgxlkSsbFzDdJXmmLiRddjNLBaJxxYYGzgxwWrKgagWWUeQzFuilgmusZFFekdHDBQYrgyfYqsuVucpFCPEIccYpdtqvlPiMViWPbkraQbtABsiqqTsanDwqxAvkKIsigyHYiVXPbTxoJDjGyEPBfpXfIeFJJtsgislHAVymMIqaCfHwgkYNvAzGnULzBXOcZPUUjGrpqsqWkogJbdKiVbBAIsIusHTsYFNQBcaSJvJRmmDenIkNRlGZYyJBSenncyjKOwelSWCPXKCrEEQgizqlbhcafhnsmnhPOzevCqIcUSEkwLCKIvySAlLafKRGCcygpIpUnBExGcTDufoDcicRTEgRJMGMqaCZeaLjgucXZNlktkBytDJGVNOibFhpAmZXHYZckTbuDZszGnNaDFOvLiqrGnjZcVDVjmGguzsQTafojORyvLLQViHofXToluJTwcksVTPILOXLTHmojqYNcbHbWsQmSBGLsrQGYKKBqfIYjGFGppPFHudheOVTICAEOdAtFvtBPxZYebdHSlSAQBWJvRiJEwKUFLscssNUFQdlAUPIpCkujQBHHEhwNfNcLOzmoJWWCqGLJHdDMKnuQyaLMQJVIWtUSEnkvaTEzURThrnvsShrcDSFbSCPTEjXAgNfXNPJFndwCsUUJrorruOUoRtdrAMbzKLBvJaqNxcpOUedxjbCNSinobUCNcNzfjcaSMnHWBcPPBdlUABKZzRTxiZDQUAkPyYiKMFOTBIsvZpjkzRYbqWdoipJWBenlqjbepoZtvzsdFeLVojaTZwmPvdCPZJlLwOsrbxHupvFBMBOupgxXjTaHISHlSumlGeyXYeRuoWtBGeGOQwtzCfuzyLMzHTJBXHMigecKVctPuYxBtqgupnaHhjSMxgjNaAhVBRFLbyHctKoAeClcQkbZjlDgPdNmDrxnmjCqvwbAvXGyOpQeXwfadzIDIYNuXPPInMDEndBYxSjqEUOWzKXbpFeHKxjvvKhLGHsezZbNeyWtqQscuEbVGOhxMIALehZTCtvGlUlYsksEDLXIBBeLRxtqsawwSHyMErPqGLavAxazemsAwEElxCXVZzHtlgMckbswTtuLNkHDODsJjDObLDyyTTiAhoeVcbejakgIwamELFJaQyKtjzmhGuJnrXJnYsqZwWycyitXnUsjxBGUIrVWHbkfbjIHnKCOrLvAvOfkOLHgAwsDVPjEnglhrTLZlniFbxfJraVNiYrpfkeBuJhbWanQrUzhmPRjjXaseCoiGvAEWFdkgaxnOmjKTcRadoPUNwMhpKsNdhfpzzlzadsVdAaAJPSgGxcZyHKbFPHghKsDszicLznFHWvjZFaDKWBMFINjJvauhLzXkIDUsybQFDyFsPjLrJgjMxdrzkarFlVTPgluMaRBOgErJRocUGWmQhAKLHAVueHFnwhLqkEnmubaCAiIoLRHyNbvYQEWbqLgjWMlklBISUgyCmhPvKnwPLUuwIzjmqIgTZFRGTqTmosbwgvvbAaBBJeJAqyGgASpLeYSHLOOCNFOmPZMAJrjNjAujGgzJbvNQOBDpJJAaAunHyeusvwYvmFoHbDYBcJQOdWHcjZbmCUkWicjGqXlZOScUnBZIrYazcIqLFOFAiesQEeRmruClXNqRiDWZXtoPfIBxApIrMutLXySgfNhLOmAucuuhsrFwgctPfERCeTlhMWemVUyBgevmVtrAImViDqLqPWoghFSsmTEokgRXcdhlyTUpjkBmBCraZvcdATaMUTguQoRnYrHGsRVTVWdtocKbqpvfEcOmYXYZQeSJOyLQzqUGijLEIBzmfUpZqdLKSKrhrnVEhRereZOXOLHtgsDgkONCxlDvpOOfqbHQIDdOkPXrwAtPDDrKXRTrgpAjSGaWYrZbTFwtlkMNRSzYPrPMJvwzfUlsWjMQLRGHvPwpsCNCUyvymYRGzwoWrBYhYKTFHrqdmnvPaqtuLrmpscoWNNspCaZsmCLqzzhxSvDiTCurvVcUPDTDchgSPrDuDRsdKSTQJjSjtculAFXMXyGKhEERnyyaLAEqlIYRlYJFXofZOJdUOWDUYgYBJANNMDydcPfXXZTSuFhFDFqoZuKIDbEEhAlwMUWjpHHBorZGmVDQuVMOsluGiGhCNAmCczGYlnTvhiyMZoBgmaulrsSOeIUhLDqZEfYeRvGHqzCTeXOtseFwwugjxNzJxRUvCCRGTYpUohhaFMBMSzaiDlDawAZrabBOaZXTSeJcplwaXfrRxHDLTgPUHtXMJnylAJmxbMeFnrmEQAbTAUrjXNYUAAJxMmCDZiKvYxRSbxeieygVhlYgKcIqavDBtvqcYFfETvczZhlCCRqbJRoUYMGNibXytyYYqCHTgKBnPIQenFaYBUnYKzqbfDhSogJLwhuuhyMGiraaPKYRsfPvZxoFUmylNyDdhlDcKtTMdqisQSBdZVrmYBdIQuPAAqNjLXGqSIYQtzgHCEMoUYjWkooTcDPTIMkrXLndRqmocopnhPCNBtbVRSSATuoBQZUcfRlkKsNljLGOxotloHYauPZArtHPZCWAuVgQRIVHnEqEsLZKBgGDVTrnYVUvcGRmMxcRsNrANlxrtCbFsCkBzQrVckXlPxxDlywIpUCeApymXGtjCHOSYGuIharvoniTkdUGxeqYUzikSfPrfSBILmikQnqZKkdutXaVsVbivcLuaXIXbvjYMfhgmyTIVapEgJiZFldMnIdgDUESrSGwCJqkgiOXSftJeklqwTuONQkjolSJWpiarsQIWVNVIYLdcLRbnsbyZIYisbNYvTyoVbufhDeCINSNJClXNMuwKLswlsREsYRHRbNjNZeBxsiukBNfIuWIlYQgdqqsGBkIsWTcbndhkzjFXahaCLLVPUtVZhFqAHVNlQHQlzSBOvNjOEQQxJMZFrTCmDXOxRXVIZiOYhoLggaZJrRZzYrvDAIyRYdleFFGRougByorHsRXQjSsIRNryXfquYtEFRSQZGbVXznyHFcdfhFItaLtCrRYHlXICbZWxtXKLvSgoyQkKeXbxAaIBzefBniYLOfGaMpsnCHmJotuNyRdjgavdfYOlpjsPaQbhKTIQvBkgkkuFYJcSRxobGprZrDHEauJkxNHggNRDYLqYvMGiLMAOLieOYTvUrutZWPmoHnMnLBElbGskyvTfbzALMXwwwXnGtBaAKRVjAmDYoMqwfFhbESliOmLTAIBfcRAPooULSoDhNAYLkEyUbbFwUqSQRmdAhbiqYzjsAuNHvEmOtsNTjVkyOHAkFEwYohuUOQJHjBPthPJyMKkBHUkDLuilpFPpUKoDsDdZxOIvJNuYjwGjMhzGrJnbsAYWjpYbRzjZrRSxpDjQYjREVeYlcYVLHftRkcRwkxqAvDwefPoqlCCFOPMPAZmfZkTMpeyODGeuxXpQGtEaOykpsTDYLRwrDCUfhrJBxgSgUxPoOLFEMuZVgpABIZpRVyppSQRwHZxcmMIVIYCaLUoRvcZBtiEzCGQvmsarvudFZgMqvTWXZMeNaOPNAtgHpUmZmQTjLwLSHawbJmnIAGLvqalOjsNnoklPWFWSXHVLFGNBKoufoQGJQChCVFEEpxsGpPQoxpcCmsBxVNuLkXlcDwWqAIDbPmpMNrqLnGpwvUAcCjcJtPRZLngOPzpKhYHFrhIKhRrClodZFnhlPfdLTYnOnkcvRGbZfIeIayPmcIzTULzXBLGfJmcvRKcotLHpnMrQtMXodIZykQAloHiaIHnHZHnYeYcGtpUeIbofrIvWTzyezctJPIZIUOEgDyuMlQvrUKifqNeWOzZftxKVRAGUuoKHIJPbGitAHlGXAfhKaOJPMvfGydOvjAurAZaVeXAiNgtTSZczSbjgeEjseBiAgOvviGUxNhTrkDkPaiAjWvMmlWVLzOmaKIgzzGgrOxVctvgmDIHBdzsMlANmhjHGOrNOgoShIZBFcIsRCoLGUPQuLQIJXpXrqyWHsTiKeEyaeJBIysyhsCYCtKjTtuQlyzgoxTGPQfCRXfTkuUHITeygwFaNcvKpBMvpNFOmEkKfMPpYtZVpMnHcPhrUlzBAwFluHHanqVhCSsGekibwxEJAHMGJrGCJXhRTOydSsBubckYTGnxOISMZzXkQXoPEJqpMtwQNBGJPeqMQJfgGYcfJhMQvKuwYsTeIeXrjtsnGambSgLuLPXjmZmIAoLeCeJfBpIzVRhJTaPDfzcmMeSplAxCMVxBDlbbyEmSXkvZyRcsdLMmGWQTqbHAuzydaOoYUMbQWlTUpZkSpWeJwcWqpUBIEpplKipTBWcgoZfQjwJKRftllWk</t>
+    <t>Pf</t>
+  </si>
+  <si>
+    <t>ju</t>
+  </si>
+  <si>
+    <t>iU</t>
+  </si>
+  <si>
+    <t>CY</t>
+  </si>
+  <si>
+    <t>CMKHTlmQwuFkpEYNfnrRMlWgDBXPjgnLNXZVLBrMYbtCPPtpwZeRPrcOKxGAODAJNFRyyvDoEdmhaSyvjhrOtlJpcGoTHOktoNenKykdlpSvtQDeBortRxTELMbghSrj</t>
+  </si>
+  <si>
+    <t>kmoYJOmyuylcVmTYhlrilmIiXpKKWDNtiSgvxxUlWQUFSzfsLbiQefBiwlgxnQClqRdkVLAblUhyzidFkFlmnybRpQPViiCRRyoRlJOrYpPcbOfpTaemylWrmJDjdEBvouialjAzPncGCYGbXKCOYMEqvbsnJxMcUOBXZXCnhuUA</t>
+  </si>
+  <si>
+    <t>KhRSNtMbULFGlZTjUQBMzjLdVLXSbfumOqiRSSwhvnMhxKKJwtfvNdGnyCZeJsZGmjgeWnQrFvzMaZhxmkCDtjbxSQGsnxYOhsSryndmYhClLbdf</t>
+  </si>
+  <si>
+    <t>PFLtBfYqVNzlMTejusFuUcGyHNFLDTQQiUdIUXuchFHvfNtNaVTYSZMTmbhljcODfgAOrgkGxpHmQYBTCRaLdSxkZNJFFzmYseMKMJfCfDjfpvNRnPjkROdHcYzDCWliEVLWrEPvkuOIKnKDssgLgG</t>
+  </si>
+  <si>
+    <t>TFnnKIgiYgHCuuqlkaqbfkryuBFDLCeZVHmdurIKoTswfdyEMXgZOmDCovGbAdUIWnGYQqbIDFYOEAoZCrylsWGMZIUznzPPAEdvfNQiWadtLQJVVLqyHnpxbneaeDmNjhASetbFyMqGkKpMDKBJXEAViIVNlaWaufyMCfHENZSuiovICVuHPrnhVYvibYZVtmAqZeWGkAgvDFxZkbvZuplnViCPsugcVISgrGbsdtQgqeLdvomndLePsXBjeJjjIWuTrvcOEPilpYSLBcbTWLTgEriikWKAWYUigxyfNMPFalSPUfYtSHjnbIhAbRWINxuGkTyfUdoBzgAtCexmJXfTxOKizOcpHUcgxXclDfmgaJSOsnIMVWKbbnuHPMeYKBydvxRCsOlSLuiUhdzsBGakjjKPOevLgLMgLeeNwJCYbgskxaxkMfTwWTFQkabHxBokpvNVNPqSpQRLciMpgkfWuUwNmPiKsTXyqwbRqAfrrHYlXWEVxbKiLAJnBckWGydpPhqpIxGrZxCdIlPTMCegxobgJXRUekImGsjpIycSRikpDIcFCXRLYTonKieIVtOppLuKRPTvlhtPaOPDTiqfbvXaoqBblRiCaAWTYxPKbNcpANdvHlMEUKRHuZAlsHXxKhDMggvqTVkbrTsMdexhyvEZdTXfLGNmHGdjesnCEtxQckTzWvtKdsTCPjnIJypxlfpFXZZnVnnElVSRVVJrrUBiDhCvsVYCMDuazHOqTGJxjorFjgmBPDQyTjkWZdJpIKvttOdAPQBChZOSoBgIIwjNPxMjxXeyrIAoKzjdXdORSHgYSkxgJGjHtSPwagAUYMEkkmqolfgXaAZwwRETBZQnraCpSqldrmNtIklRYEWJMBpUaKOlTbDPckqpIoZdoaqEkAamdezuMmzUaDBLhOYKremghWcHlmDzYxxadsrsVbEdeKxCHdbOLuTWbXKvNUQgKHRdeKVUfSyyzozGKHjkRpANGghIxdcbVYCYINVVvReYCHlXJKYFuCNOBeYxmKujXGLEIQBKbaydOLuyEowROhIzVdXwHPpACWJRzPOUXavyapHZeWOvaozsgphpbQFaCqzNCvHAoijJUHCTAOEXoiMIYXBvmtBtoEzUSxlvhVycgCjAcXRzpFlGoEZAXSKMHvgZHLeHnKRVzTzXcgtjigAciJubivqHvcDoONhQnHIYWMkZTokyaQOjiXbvyzAqNrafxAydbTZMTGalamYpeaZioPkNDMEbzxUVEWPpSrEZijLJUFIIVGMdmmowoSNgQCmvhCVjTMoXmvtMGCzJDFaYugMhrYJYjKzYgWDaSMEsqnXtfEvRnKrwyHmaKZGHKjXCSEDnxKfBOatxPwmSUyaPnXwepViqkqvYkfDXOfqpiScafapMpyuEfsjSYeeXnJSzTPtRdxPWxbPELqPwOHtRBfmYuKaDxUOUJZScHUvTNLqTpMXICwXVMFDzWYRatuDZdbebnKNbAvckLOrfmlbzutIUPlXchRIztQkmmteYWHvPrGPlquvtLeIcncjAaVImKeJKHzRTgdJPnlLvoCCkHhnJAFOGDwCkAZxZTAndaQrkglObhPKHpCusPGDtahfKdjMLIvWqOdrkRMWbxlkZLeVMrIFQYeVMpLRhuQpPuRMcarvqzryBODtKeOQyNjlGSPcysWUTQBibWZmvPFvKoKiSGYdwETkkfwVangRdCdFbZhepqAQTFgiPbJCZiyubYhSxEMpCXeKzJzFpLsZTnEgtoDDWJUKVdxklBbrLvEksVjgeciQPSViMtYxsZpBYFqddaQxcElFnPWesuFLzEOqFSWDgZITpdaHAduuMOPEJftRpKOzDHzlXRRZJrIQFqILZqPBIvxYmNGadbqsslJMPmFoDkATxdxPxmapHLyLJVwfoLNGLhdQEGSLVqGTbJVoVgELCsBcMYSYYFCRqdlSbTJTGQlBpoManYrxTgPMwyxOaEbOEnClHIKcoWesxuMyXAvGkeVFrSyLGtZzCgRFtovFUKCbpRuBCjMzkhUxsoFKZXOiDyDLznoKLNhIcidMOsWNbJeeQxJfndYYxWwItworwYuYqLeDAbsmazDaIszFJuiQeBoWJLRLIHUhJWhwCdTLDOrrrtkHCRqalzprkwvzKRBWWWvKNmjGrhjCBsDtWSPvsLyjHMIByDHdPyyAmuJbfiaQhxWQybTDySWLMPgazumJZGZjiAzbESTqCuGzTljrZDXvOZzulwncGcoCIcAjiYOBLEzjjQsXvWFWdUQaBRXyJrEShkYZXplpttaVuoGYDfpGssZDAKGyhIyZxmiGQucBHWNrYgjrgZYMyephSPrhRZnviRZzBtOCygaWHzILEWmqqbTRFkUqCQUGqrDVbHNthnVAZzvBSqwvnzsTGLyWOMRUTZTTKODEfTzAJCvPftFWSkWiicRjZtrHrhYADJJIjqbENMaWTSxqAIvJgPKyKYzlMbXJBwmzOLyzUsRVlAXeTPwegvxlKdrEzpiVsZdEJBMbbwFgtsXvyzhqNPsghdxLFRlkGBQVZoPaThTbxQvvYJpecTogrynuYxjZvTwLvBAZAAeDmITVOjPyNPNrsvoOJohYtpXoGxmMWxSCqCaMgSuCawvmEfBCTFYbXJTaBMcoILmjdAHEtWpEeVuLuOiPinRoFnXsQMxhrSMfNzKbhpZwbptBnGIDNrQVrbZlpvJTvELJdYHFPpTmfFzehKeFgmVpNzRWgjlYFPDRbjrfqgVgdusnZMzPkLSwFMlDMmtXdsgaOmooOMxsNIYuvDzisEXHKonUIfyqbSQIuowoZCAXMwGzbSALtMlcQBwjWCyspWZZwTDppoMzkHOPzsBUIYBCmIYyBdVYkLdEpATMWNYAqTxkjKMiwHhfjSIAGaLiPuRRoAVjyErsxUGLGBqiMIylMXbpPMtbwyAEnniwzYkoSequZGTvHmvmlexSAKEbbnIyxSIIzAFckFCUOYUAMDhNyvdiuzeTfalnJbyOKYBzpffuPgwzEYkVUBrmDKmRnaKjzgfApeyWSxmynshSQiZNLLxmYmRoZWoPHfhsZhnUPVFKFThQGhAXZisSxObzCooATsvJANXuqKvQIkloRJhxpfIYAuBUnrbqhRcTVCiVNGVhFImxlYetnTMdgYlKFglvTQnefYYpjdMLswhhgXhXQcUGMuXrOMkUJSHFbWzdQUuoSVRpNcyoOTNmqiHOsmrHcapCAtSDmLSBNQDnvXVGFgIkLmQCPfhgHZRuYJzApWyZsNxvWfAxmmEGeIUlLCgWAFNqYPcZShZlRqEAzJmGNURqrCWqffsqxZBSasXffTxcBazosBNaheDjvhqHZcRuLHlJWAeSyFBbOaIWLSqYcgkSlqOlfprXjjSpxRYwZNaJnwLtHfKTabYBnlNhIitVSrChWOtcXqnyzWpVHRmaierioruJHYmYAVSlHoYNtsMbnpoSICtCVNIHzgSzPtVwSfUOekCPnTWgYQtJgrHDlYUFTeDuWSjewVQwrKDPeRhjFRsRpkLgAVdAqlltpOQJeHCAoWtVzmYZGDRyWICNzuWZPzjvtMqcVDUfsvgBFGTiMtKeUYKwAaNVUnVlQIxTsBkgJgCpouCrVmqztHJUphIHhhQkkGUobPFJvUTsYDQdNGCRKqzNCzZqgseRAOfqGJByNgYWjAUlZogOKralYOxMLZaseivlrznxUBIcRYNITwYQgnDfhJNqPBdufEpuwLCgQQchDlyzPWOFsydaBApNJRlkjDcEcWJcSEHHnRyzeWyMDluAMUMoXVnEdNtdRhJOWJetNlwpveimLsuLJzddKUPlMqIgmRApHRbwZdgnCAuRaeCvnUbKoPAioKRvrpMKtLbPcSBzWnIEGdaxIUZxzZwjBnHVRxefcuwScdjmoeCTCyFVtBGhyFmNAGQHOOOBUBXsehNotfWCeINDPTkFmuWjGmFeNqDRRPKvaNhDtuusCPKBnXwfmkSfFupLBMSkPJyedRjAXjzveNnXtRVfHsyftWOzvxAseqwBAZJURQteJJkxepMXbaEEsvhmXsxajyIashUWyhdVeQDJCkVNgAFitVnFIVBlTFRJfOgkMgnjnhTCqbrQlYTTEbrCSOlRSGxoyIicLDrELhPpuifEUGCwhcOGIPbsCDpzicPSPaLeuRlXBKltiVTRZgJJKmUlxxGTkwibsugWYTRiXWAOoYwzrBHllqXKESvvjfoNpIQdBCHGujLFMIYGJpHEBzHmaGbVvvNixFXzRnSLTeKXAjnuJcXnoxOWGwdblUIFFRUJtWsjVqhjxGEsxCGRDHHqhVsuuLFpkUSSoxmtUalypZRcotwinQcMbSoUIvfAYvqkldGCqSsaPUwdlFrwJwYJNqwUEfZhNvFunjMIzsGPiaQfmVVjfkPERWXlnjFMSialKVDYxKyBwfeNnyqqhHgiocdXYRgkiRSJNbKgohdJkzhTXxksoioCzNksnMlyFfgdTmExnQVylrIPttwZwOIoGxGZffGiCZACRbaPrGNpLbPynaNhtuwPvsJzYDGkdUgtjExCLcPbwLOxFiFgszdToNIvsilixIamUJauqXVILzcvDkoRIvavtOMlJfJOZzXKmRlkLlfaexacWxdnbeiIMgYFrPCAonlYilYsmgVNqrlzlePxNeUHQgVXljqQUHeQQAWzgKRIdvaKZlnUUtSgAOgmBcSLppYJymxwWdCRqFmduFdWxUNosAYPeUAFkuOxOMVJdYukxPrLDPpcCRRoLNINKHbRznNEKjjwuCTOwBHSiqPwFtYxsUXJXhWTgPFJdkNnUZePijpFJdpsNAZGrnIjLgqjFfSZUgmkabEKHmddJpPNAkshoLyhJQvFLliKgcaJtjpLSBRNNvUPCVxbJAUMvWrnwAHdbxjmFMClnJVdZasalUiVykFGxdnEUzOHncHRnOMgjWwovVWMkBoMCqimnLxoOHGmLfoeSNHbJCBkIBZvATvzqDwjVxrFeKkVIhFeDOdtzTZNjmBDGisKEGRmELToNKusibtUShUoWkUDwuaTVcaZfdIkYxtHfvaQnUdbyezPumfSUQpaKIOoONRHVKoMAdAdTRXQulHyqxZAFOpicUqyFcTvZpuvakENdyREUFyYsaEEpLtmQcKxAUXKfhZotpwmeoneYVadwQfwxxOPTTPkCNkObvItmMMOjWlzvDDJOpFoIxujAhzqrZnGRhJlLocHrospPXxaClJgrmHJrUWcmtOBWhiAMUvQnfNzjnmmHaOkoRhpIgmkPfzYEMAZIekcuzoBLwElMxIISYCDVYZOKCJWFGCrdiCEmqCxpgxcHKCvNYhdcHRCEMFlEZYpYuSlZDRRclNvrqMbMQjdihDFZfFJVKCjweannEQWkFemtUSMpvLltrlBmcrweXUxNoesHQnnEryXNeMDzEwhMnfkleMxImBiFgJStrzWCpWUWaYxvTkLrsFZtdSZWLzApVVPINljSnuvWlRVThhaQPdXxRxNVPZHCLmSZVoechWDvcVaMHfnKHYGhFWdUAPOTUgdbnbxvIdExNZySHQOrRegACvJDJRiYwVFrITTFPnZvzNHGbZOXLaIoKZOmGbNjReUehEuDvCKcSTBWCZGPPDeFrbnhfahLRxXQgqBrFYMLQkaulWcvbFLMgjGorTijlxqTgoTrdpexAwgrdHGvMZdkQoysIirPFqXjNDCNoVlnSQgSjPNurfSirCWUVdyFNzbEnhQFkiWTbgzgyooFqerDvxnoqqgprVSnZHEOpoLoLMmnWwGkVfyxXzzIGzxVtvnrSwMrWyeZxsccrzQxtWWVqpMymhzcmhBNlmwZBMgjFAwewABAdhbDlXUHRIMghVvISrbtoqfgSNusYNovjZtWwnUYaZqhCFjzxuAZQMEXnvPjfcXLxOQBbVndVJVwFyCZkiDLcKzvdjmwwgyJtcgyUQRBZBAOdAglVevkSADwuVxKfpoLCuMCAiyZPDPIKjPOgIHSaZdhdIvmkKycLzsdMAUzpUCvQjPMTlNBYErlWhUhPFPFUDCjXspROXXwxOfFcnfkolRrUnERlBETNNkcuCXDwevBngzPoqAShIanxsnKNyzUjNEOrLFKHBLUIwIQZvAdiDQExRXqQjvGAZhkMtlCQifNTReKtuhTyyBVVcnPhnRfNJPqEfnznwXQaaIJHypkOupxgOzOJWKuHhylGcmAJKUtWxbwwAPpqoFlmqXyMXEFqyBfMBDQULeAoMPFrxxrismiHoufgOGKsOTtyUEQFdJBtQLnOsoLhZRQlSvlQxuBUssyXMfowyJOSUAPyNwyEtYENZiOrSJDQAYOinOJwDiWXOjqNKDrtqRUBPQAzxlMTWnxKURxbMEiYdaqvWoREBJzqpLuAGmhAdXoVmiFHArDGaCCdhamTRdsoHVbKiubGjMKZCvkdxggMnvijVrTLzKXsMBMvSBoJwRVoVydlgJsHRrUZCvnGBhxDOKepuUhwyYNCAJSKHoaXyTvEtuGSOnnUfJkksoxGFlgKhewPdFbzfeZhaDMKwOrmEbCwmYTlSHXQuvFuJpDjQrfzsnImKVwisKOLcRhHVVeyftkiWmjRwqjbhhUXcYVTrYCQsZLaWMdUOeDNoxvRDSXvrwETsShhArnlZkcqKwrqtXjvYFtCKkNimcTOnQgbIuYUjlNTRQFpjJSYLCppAfkllTXNKBOoAHpSqAsmYqvPLzVGzEgdnSGFVffdwGACjhBrmfVUBaUYuKhfTohdLQOvQmQcYBFqoABHHIHZaJxqgyKRNEIsMTFqEyUxkaGGtCIwCswABKoIOguklGmWKnRBeYdmdmBwbSwzncTTIVmVxhjQIafPmdecXoFoJTQynZngfzExNVdxqjCVShzzJJCfEgoGcpowhYCBOsFkCNFghxEPssAHIffbmFAFklodGHHMuwcLdMnCcoBXYDJEQmAxwBPesUxdywzGdOUAPvqbskfGPTgnjDsoftMmOzIMjRkbNOTbxNWiwTZTvLcfsMoGaqeAlTBMLDdlWcWyfbzgEfnanfAjzNDaMyuPDfEmZAVecgSkrhaOzTOIFsGJHIWYRCkdcqBTDcRYAjBKOvhLVssXuPEwjIlemosJQpQzRCXtAjcbSuaIgLIPgPTNrMSFwAZMNMqlqRjsrmZvToXBTyWNQvlApjHMBahJKAOAHNfoKyFLQWfbfgPtARcBsNRtbytqkTkDhwSZaMprIvkIXzzbGGLkBsDxOZBIPGgIRLdCNaUtzzWDfEEOVDGsIvZXNioSiplwCKCngeKDJKWjsixsDtBMobbdRofKQyHzzcQucqAPZVYTwHGULzKUymcggybYGUemywRWyBXFfBGAwlCTXBzmmxNDFjITUyidVUxqmkMsahVNCOCjIFnChrHqKIUGiSsLGYuqpAtZWJcedKDCsAjimtVbXhzXJTlphHDTZDUGvNmJVMFBVnMVJZJEovjvezBiGZuGWjLJjKKXAhXVYpTJvbSFutdgRWwqjNYqSBuRLQHDRiZHEFuNyWLLldYknAhBvwRFhBfOZXfSBiSBYqVmEWnVwrzdBfLdYKEKfYuERAQrcLfYZMPGOFVgsvWGmjyfMrFFwtOBEAvvXSFrUiUOQHbIZuzGoPpAeZlqPJhVVECIdevguYaVvkyNFYCKChLLqIUHSXhlsnYIFubsBJPbbvwvbnJLyRNOaixZaEHFUIgsPdHZlARFbYPAqGaBlQuTUMdDlVKVkWgJFGscVeYwWrJOJawiDJTdclMxgKvGZlGygcxXsHVYJsKndFgdkuAznBCOMsFiIgyOSkcEFIYmMwRbIAGvWoVmPlCkbFISBGUEwHPKFefMPKAzdLqRvwnlCsvswMYlhADqmimSnynjzfbTDQzrUyDNNmhZPjVEItvkTrXricFsnEbRvjzNlKcAfEMfHafyzzIhCwFMzqFDGHFgeJWNZRjndibrzjmIusYSHeZjfTuOUGmYFWEJHUaovVFcuEtxzUkFFSXJXRRUJgXYbHtXzAyolBdXDlRdRPfmTPsGrnDhuvALvOEbhLRgqZvGMLYUbQCxTzZYnJKEUDvYobQxZghiYPqdbjcnakTXeyWNEvpxAaiXSkEztaXZEQWkFcrdgBhQcQYGPxtVyrOJQQbufflFzJzrhlKintneiOBRTFlmBPzQITcXBTmfvewdMACSWLgciYsvFEehbgJoBiRBFPqsPgqATiLQNgoIrkuNoDkCFJxGkkqNMPgymlTOrtqGGPFFAnnGYzOJIkNUDrEwxokwpoGuVlDPTOCurwOyXmipgXSAXjYtxLZFLzgezzabErUnaSlCaceMCTXaaTJFNLvGUhaFpOrtUalogAjJHvvcPVcQeGNNlZqpCchKXMQCuTPfGrclOJANViGKaEvSDBFlwIOqVnUqeHHOxCfmEDmDtstHOSmfXNwXQNQdyTYBZwZiVonzkEmsHcXUEAgltxFxjhPpooJBwcgaVweHRedtmzrYIcaXiKOhjVtwdgVNPDpipwQpkikePlOlomlCbeAtPnyiKXvCmvhulrrmUNBUvxpWiAVWPgLjhlPrKTykFQCTUTLLCGZjikotuMxsWCcQYzSKqVHslkNaMwphxenSQDyplVBLRzDEFhvYNJcDrGutvtcYrkCoaKcUWyhOthhTHERSwnGErFgFIzSNIgpUDTqkpfMKFnRlKZxamcPWjgjEdAqManOcCYxvUZXfpvtBUYRmyyDzOjjHVMuMMhTXDmUoGzrILNMRJpVRmrwBiVBZsejaHXipgZqvIlgDmeKxCLXIhdVekFJKOMKIRnrhFHhpKRTKadTaFdaDMAFghHHiybzHZxxuWGENlHpvVTMVshEvyiieePhhtJpVGMnwADBTmFetvYkvnnzfrtwcGsQMwLzLWPfMCqJLucfjcjicMyakdbrpbdXTyEBOKKHhIPZclwfMXbDBniRVctPdURJtlgPUZRedbgwyJtlzAAUJbQbJPaXttEGhMvEiZQtGWPYoSPXjemKmMInSsQGksBjaXRAuvZrPwIfQEmYGlpfRjPyJtiloPTkCfudKLpjarjsuITlyMgBjQICbDNKNFVKhpSDkONaZSBRyHWOVeBbaclvPZOsXkfBMItiQsaxlwOoSNwfKPpozdpcnutNFQkrVQVwpzyvyqXvkQxYLwgxBGQUjVHWLDcDZmCIYpusPJQFBXZgtMHqxrURfBIgKKpEVSjMqqOBAhdTGrFvMjLfszBHyzAxgJbdJsWuLFAijoMMSKzkqIQeCOeNgocdkbJljatYIfFFbAxiaXXkOenYyEngrYFtCKmvfZvPKepLNWPwuXdIusmZLNWyfcrCrChYLRiMaWwqUKWOjcVcmwnJcVkJXIvBmjcLHNHqzAHdewPslmkqbrPQlEFXBXgcUWHUENQPVoiqGBsNELcmYiuKjnlTDLfLkvdPwnzidqyBXsklKQgiuQTICIdhQSBszUdCMJnObfpDOqDlkJDAYZbeYGBuZeeMsEcsoHLaTpTGxYHpLsrJKUvqYayXfsaQUOUFkVnlOtISvrDtIfVtVAMBuqWARkbRuoJjeXSPrUBndyFzoMcVhszaIqCpCSnsAAYfgZOrPKMEHlFDNyOVnroWsCKFqayvbmTMclPwmrAiiqMyyLNjLtoEdliBoLNsOKLvwozjVpgveptvjNKbYhbdkBtAsSnQoUnryLyZQQRMqYkjgQhMEiMCaMVLgujkSTJjadZXeqvwKhFpjhbklNqHqSiyCSNyFXbvLQZBxcuIDtGCSsLxIKfSKTiotvsQqbVkhugTUkDqjcgntEHFyNVAqZfxEpTtJXSTOKpdIDNNrrACjHiLiNTFsRIDygkCQRmZbhTvIgUCAvaDjPhrvZiJqcvSYKFxEldBxRkLBOxWoYytBroCvnBZGNJqGatQmLCQBtErEQINTkHJVuzQIioVgyWnKkHPHqOGIcuULvLMTmfEnpdMmEdNwDPfTAITScNeagNcakbIfWzAxBHErSsMdBXXEWbNFvlqAWDAPFtWEXkTOnTRTeWmBNKckiggZOyRgbbErKgKmFhFWGdSfDjFERCfNBSSGVuHSQWcgkQTUrTwbTSbGUFelOREnqoNecGYiRvuOcvYnONTXnxUagxglAXhUTepCNCtTiekfAMMornbbaXMexVvlcFcQwPvzUAZPBRvvXRohqNNKrJkNbusPbEvgRfGqLXMUqHGdSJDfplSAevsraPyhmZorMGosDKtaIeRGvFWragPPhBkLboSqUAQZhIKzwjkNxobrjJFEKEzYfWpmtXfYFNZKnpplTZheQdVRxKTMCUsmBCTGIXNcYLewIibvpmjMiVAQBtHmqGROiJTpjGXGURPIgMooNBZhBMgHzYaiBzeCyclSkrCppNWbdMfkaHwkUwNWpnoxbkEcFHEzYsUYNvZPZPhFtiPqurCaGqsUCOdbhApkppxlgjhqMKBTMKDXiwidhEjDHMxzKgJULjehZCnBDzbYrOolETrVgIIJGLnTRVJwvSdIcCpWtskFUNCopXPGwdKpPcGkIcViOaLVjQWUqjaYNQOlFuOvYDbbKQRkvQvTByvAJhVtADXKFWpWhUejwGawOAJfUQKmaoxfrFagyvvhVNoaZSLaPkPWgtMhKVpEvzRTLLMxMwgGUBrfCEXMLGmtcMAShxItrOgCcBbpxkmfZqYINYUMuzzWHqsglnGlojnKLLRWhfKHynjEhfowNlAtUMnYbexzbOTwaeDaBVyrEXuxbhwSpylmTpvxVLbZKSlSsPZIJYzlTOuMojEcBnvNwFrTRhNzwbfJjZWTQIoqDMEqOUTgKdCLmSyZHcXVZZMyRgBYwHauJyZdnJdVEqkHnZGEyGHMLEjjrxnOKWEmJtcowYUDsxtQKydHLIiRWdGgTjACQtSuvqMWcLGfVKlxyGeVntjyNGKGuihTuILSrHhngurwaNRPXywZteDIRmWDgDOHVHEQnyZuxnfRAvxRTbkADguknYgDCduCWxoOYRZFKbGntaTBaeLfoKPuHevUfJzNjtpnfYovdhLLRwPUxpLwCmPPwxOfWPtJPyDSbyFGepWmvLmbWLkCPjZxiZlgYAYRLoCvaBquEcwLCcIUZpaIDEwpytSUSuZGRcfRAPpnSjerzASYudZiUzVoJQcgRNcWDlUuzxgECNdRqongoxAdSBukVvXXJpYohAhaWefEVmCGXhGTQFUqSTFNmgPtQrxRGutHlpuwQowdnWZtwtRqZWjgSRDfKFCqDAAZnRVxueNgFiqHifIqNVUmAMlwKLaazKWQADgIRRcibrkfAjiDCxeZSuOjgjNYtOzgmRTHuZTTuZzgZYTzTOOVJrRsniWDuChTMyfWAxtKeADvpVSchehcoGqqBLJQmtzxIZJcOJQXNliVRvTVpctHmnLALIeknXlbRNSgwhwqtRJVYUnOJPauqgZBTnpTXWnRSXFhlVupUZNxlITdzrJFSnoyysLaahfOPCVlGSMtPTlHkAOJBjIePpELzsaxDCcbbESUzeySBWeXniOpPTWZSwcrkHZcrRKUEnhkmDHMsBoTDkPwkNPwyqGPaepgPVJVvKIidicHFDPdSqDtAKSxzUyTQdJAeDBVSWMqEUIRcPfeSiKZYgYhGvEzUPTyBnAGATImMPuTrrGOdbGcSTGvFJVehABtPbLmXBpfdsteInjEBKiyICcQAlyaEcvyaSECEsQHVbuwEeyJmybAXkisnzQZuewMtquxCftFOOWmhEdSXkNIECPZdpUUUYFUowNbmRRJUvtqwKVByBlogiQBOKJVrfwtrwsYqkRBpnNElGypDQICcwxcCutsgTCzhintwjVpsaBrAsQvUVmYUrrmPYwiLtamoShNpgmcXyoKGXtRVNBNZWGxsaCXPgelxlYLiugXQjhmpfyHmoXUYbGVtgUUIhjKazpaeILvVMYIklApeGwzrurBSqmDYKiUlVwpiAbNxelQVsOTLoTZGmYgjyPjWQIFVSyUQtswpCVlJiXUCIpJQiRHXmaslFfRtPFeUjNaApfrWNYpUDVAbCATItcqfsweLUbyOrvDYuWuhhmHtuxGAJCZeivmgACeuVItbIfPNHvXCIsGmMXYeuvckaPfbLKCdSCwMHPxTuTiVIBSbhMDoDkIMDoqolgxHRKLkulgvBhoKAhUQpZWMGeuGKApaWsFUcJrYvqUVInzxkXIbbiGmXcHYwHhlkrfpyBBbcrvBFrzFwaGANxsikQJhRopcxwpGZlxhjeudXoVuZrguooememXAziAsKjkzdzAattFDgGvZKjyOluqcwLziXqYYMMChwqgmQNhiNoZphiNHVYCAmmGsyYLQCnnloYZToracfkVfteDFCSmWPqAlYuwMyrseBZyySapxTCLTuQTsfpcSCXQeIYgGoeHyNHAllnMdEeClqxSIOwFLKbajocoTecKyXDztCLKKsgKkKfbtNwHJFoCOBaVogMJLqWSBUoXjYcbsBkONKvTqbwMtfnWIRylDgdQQYOhvJzIAiquyCUjlQMzuJVtnjxmnEeuiLqRhJrDlQxcuLOSEUppZElrKtybeGaONzWXmKaQHoCMlZQNYIfaeNcaZNEojoSOQjmPsoPWyzhGWPsclqRJokrtLUWxqATmBduzaRvgVtjWUvGUaZMqDXfOPqKwAzOWtmaUIVjriBagOQDcvpIFXzWaVLPKeAImWwSKMJWeyFwplgboJduMysbcAfmJhRYgSzwbgHmXXSdsKByJLHlOxxOQDAWbaKuMxgyhOukfwOHQkFpGJFnbguEwUnToxQOruXxrwcqxruJzMolNyGnGAUbgKkHIZBeQIliFQNwkUrZeJGFbfBQaDpsUfdkYCUQtihhBwyVcuAFCkhjFhNlzCumFYDoDozttCiaGedSRcbDIgTepZXRABaHciYhUfLhyXjyWQYrqdDvKKAiYhygYlXHcZHHRbwjeUgHuRNnjXqEzbqxieyewLLTmejiMjlztNrNahxqVHrLlMiQdKSUzYZKwawIDVMxJyhjJdIKTvHyqXbsUKYMbbMzghHygyWPFKzOhjZEXeFZQiXvrMzEjoHPMInuexjNWxnzDstHZFHoqRaHHJWTCkmzZpHMLdhxPPQyrIjuRyVRUpUvdydQHKANtVslLcgdYnPqkFuiLHrdUeJllFTQXbOyZCdJhUfFOApXmgoswPTQeTDZUEYFYHSQNxdJLWyKVdLjFbhJbqsEmoFPdYHFdgWqQvYHuxKzGKFKNpYdtwhNbathFEeapLmdDESWNaxxHmjexYjzZBPnFeGWWDwztiqoNHwGCtdfRYdsAJWCacArQMIkiHVQmVmfWMkjdCCDNpAmdPyDgrFdRCUJsmaYOvEedSYkyFDyaBjBPAQiXbnJfSiUkWnVuTVXXiFebiXGsnaYQRSsVttkHpIVraBALJROmwNnVkGTLvqXRSGHyLmbszmFKRTSRXPMBlNhJYjRdVwXPuFgvwlnxlhxuaIBlMNdAOoTwfGeAHtxTQFCKJdFkpYNGrPttBrRFHwoabQMtHLAejGakHEMtWwwJkCVYRIPHNKQMoYTpOypSyBxXRmjyiWLcsBGwaDTjhFkIYAjyXcnahQrOYhIVcpxzKrgMCFORxDwoVrxYwmUBwNRtTzmnjCCxfxvoNinEVKOGlMyEYlEVDAdoWMgWdxMGkosNjwUChDAJdpUoGOXsdVzNDmCfgaXBSbqSTLzYsLQHPLQVCBfOHfBBuEiedrqnnPZtdwcqzjohjtplNDExfhbRvLLmVRqcjzFnqQvagugJMcAcGeKgtddUKSesAsxpHcxUAvUvwgtqYLZePQZuSdnhuMeGxDkQNNogYYyLxfymxrrzTKUQVHGJIgIgHwgXfGBNOlWoPtatUYnfcMZmajSLfjLdLUdfbXcWXWVWFVYEVxJuJoyNXZxaFNBozAuHamgYtDhtGhjHoJimzUIZzTzSoEMKZKBcSZyPPmlmKZaHTJcvkMKHemARcZKHThcBmzliXTRhcdJUJzHhruPTwEUJaGZncZHAludfgzfzSMOplCziaUORejpLXVzCXIfBLYDjDsexeZoIPjDNTqFuButrZQXSEwgmfaaAVQIuiyTCkYLPRLigLrzPQtfYCjuqYGCIKfaewFJbezbOiRdDPiOnPUgzCjKRFaHuicVrDiMXrmAAjtYRdneIigfdfnxOhbYDbyilvcPaJnmUKsfMUPxNeUvAxKqThAbGjBqpHoWGersdyZKtsuyizNWSUCwwVBTJoAQTyneJoEVMWtoWfgxWEfjVnpxrWZuMBNBlBVyqJVxVXvcKERanXmaTXiPByeJdPaWmgufhIwzDwgbTDfKmEVXOGPuBlcilnGrgppQDfXPRkMrahJqsLszLukEinhjEvYqDURgVgDhxoviIfRTHHKEVlFMBXOScebVspPjDmaOprMEBqbCJudSskQvSmNjQuJtCnietOFKLcNAEKeUCKMjfxKvOAPRcZtHQmagIcswOgzoFDXaIAgaWHxNvsSSxiyEZFUDAAGAeXiFwnqcinTmwquZMyiyBrCNFaBBsNJpIgZnOjuBhCydWcOjdFzxFrPpzvMhYKjUdYtPOTvfrhkqCnKZatTeOxvnESOJtimReGICJnuCMJJNtVUPnVmLEVAAIQFyuZLEIJpgXZgknbctCKBMkGQtpvfSQnFltJXbPAMMpgVTcgdyPYJmLqNgWqDbkeZEabETsjtFxfUdePnGrvTRzRWqdknLWtAeuZZvotbuLXJRNtAgcXdnMFZzjFPrsXOMUaNwTpcPZTWAYsAXfGahCrvOPsXLYZbJWeFDVGnCciOtScvkaGpUBZAdvkurrEFbFfMxtGNpCUBrCuwPxBYRXEwVhDdqSLNWYGaoYjutIaVfBMCkjzhfnhIKiYbSsYWxlsZxgVdpBUOMIaMpPlioSiakiZufkAOeOqAsfUXoilpVvIBAKcMwzrehaxbDmqqhoTMTzzpKOcAjugUgnwXQseMjFrCiNahkKgJEQvBuapYxRdKblqbXkvoQYisuWDDHWpCZWrRAODqgpjmlUMKCGXnNGZefcXHjQXLSjTfaLSendjsVzBtHhNQQEjWwyAVTFDprpeEEHPsWkEZkCjzqYMXYAwbdrhFRSKFLJeJGmnqjrVxLaufQCxgPANcVRysxsuxIwmZkrmNDXgfwcWOStjBPUHWeYBoVzKPktzKyzIVLmzgelEXTscZyiswidzoWlwripFbuOFLorDhchpTGxFhRLfAOwTZCCARGhQFIaqkJnMjmrwndhWlVzglpesjZFGtJxECPBEdbBoXenWzQhGlYawRRvFZazGBiPbGfyvziIgQHVAsErNKaHBsXjkIZuRHwRUrenJwRkIhoPXblPjzWibxvqdgoxLHshCmWNZoyjiWDESmmZEZMVYLuaKKLvxbfSHCXdkHNNHwYdnqLSxxbWCMRJlIJbmGKygMOMYJCsiZppzjEPgNRPxVhBUXkUkgBnPfWYpLWpVwlaXdAsZljBHAnYaTYDWxRwsfLwNMVGFhRhFCHcBCYVNQxOVzRmjWYAxRdQbpMygEHxKuuXSIIpzWBcBtndHFtiNStcbOEOkpsoVIckqYoqAEgJLLElEEMuoKXRcEmrgMLJSytkzmAirojpEfyhcKdSDUszmaAmOwZNZcwNVbnEhjbPWpNSrAIfBuDuyvJbLLBUbJFtQjEXZcmxJlCiuvTHJVdNWRmCcdZIysXgegUjhlCUQcaCenKMQKPcuDGiapRebMxDYqxBDHQqoWZNoSuJyGMCcCtPsDcwTKipGGVKNdhYkpVKyUZFgqfYoZqonypJAuUwdCMgLgyoiEvecHcVkbXOoxlNBSdUsVdtBDgHOdVFtQPHcjiMXBHHldqlQtOYPteNJGbRVmLMCLaeewpBsOvARYpXmqNDbiwhCGreTgdMUkLYlYbFvJsgsyOAJysfAxWABnxcubZGMpWcTQhlcCWrqFTuCikmXrGdEcGhTDldEJKHmNZqcSGaHpQYdLjGDjkqvGLBZGSPmJCRSfsOirmAAuVCoEtRwzjMuUoKtEYEcPsEXSbtIvkxtBdGjmhEZMnJZJORydNSKuWhSTnXuHzGiYEXmbPXjbXMtSIMHaiDKNZVOmVcYnRDTxBDobInnGkPBCfyTxwRtxaGUEHzHhqBYzMPozPXorGnVxwsEdEGRmzlaSWEvWjofPvPKMkGezjxIpczCpkqLYDzaxkDxRXPfJLObAIbsfKkDsbElyHoxHmNqQRxCiDPdipDxmOaiVJIcxHEwdBhvExkhEpcaTILTfZwTOZedxlXpmdlqGWmpewZgvSkwHFFXfAGGJLJxiedwRfNPsEtqOUlkKcMunssFRYZfbpuGVxaRQMQiFyBllAodylCEjUwVrMwrTpcxrAKntytfodRqjgenCKMbSRFQlrmFslOneGRhzMPdIXqZgIFpGkeHmvGCJLSzYbSlBhJfCfAzbkajZZSzqAQqtVvXmcIZziURpnrEPLNcvUfuXrRxMVCuHENjTYbYMRrHfFLSYSapfpRrwJJOyeigUEaVSVwBzNvCRAJmgrlWlFClCRiTHAWXrbEehOQvqcvMJLNsPOqPTBwSxYCBamxJKkCWnZkDasBqmWHdCCHlsaVAjfqGtVeIeJXlRiEnWfJUGYeuGGGxcKSSyIZsSpUpxNJjybOAFMnquiHiWWrUbgtIyimQWqHvWTSxJhHvzHxWIUsElVWscLOPhCBvKWueEvTzLkYhBaqqewCTTQjnzxDPoPyQhKtillfZhJIyFnCKSGDcXjonjxQYDYcIxVVnJHnozJgtNGtUcBwnIQXSOixfzXBqhUDSLCoHDXILTPprdwsRBUMoqfGGOnOuZcvusSxUDpNsTeShXWAIFhixOwKMSQfEVOGfXWWGJyRzFelrLkWmXQqKAcLLJYPbeOdZDzZuHFjEiypDbzRbRuWwDkZudUaIJrWhTJqiacXALlgaAslKeZXVhEdyuKjvSOsEthhscvpFgiasyadzNFzFaVkkMWkoCppNthcToGlwDLMYMvcdArxegFrQqkRfLnfdyBttAxcfxFYafcEJPLrtgzQgrFOtkAAKjwONmYjUVIHGaKRtofoeaMfKbZyenUEkoKXdroDJJiWckhLSoyxKARmiNSeUrkLZCIfmkmpYzJnBwaPGUvJEjdCBhwJpumfTYLxjkNhuNGTkBfxxoBYnUhmfxdkcAvJkQiBNMquPyoPMKPEeaGKrZIIZxgTsCidKqmBmABgwZwclvwnXpyWfcqUHyUUkQgpaWASOTkvJIEKjpNvfEhNySyMUqQtvqSTFkoZqisLeWbTAfqJRxcmjPbfMFYGUvhjNkNfVsqtACWLHYTZsuDhGHjfnZeEikeumoUVTVbLxDeNNuFFgCYNwENTAIQEqMgvKgWrBCdEkXZocyQjTDsKDoBXczWFuywvbdserfmbBdaTWAlMIbmuFxPxZyDmZYIBEDgaBGNcVzHKavqPpeHyrsMNoYGUsAsSQfHghOyOukKVEKLYJydAUlilGDJGmbGRpLvVOstFFAmtsyxezWAWdauXfYCuTYBiTlnFZgokIVAXPbGrZbDuCWTyrAFAvaMaYeqwKiGubfulKLZrQbfHGYPWItwDLuJPwUMAqCUtIquMpDjJgXyhqNhoaHCDHcbgnhvQPCXWVnaVtcIQOJLSjUDMuCzotrcicEaOvQXmdnmxGuBGlKOYbkwcUAvsakFQFBABfmjwhePrqjrMYjsoohgtqJpTjiWtYufsNCinjVMCHwmyvHibMrZSNqtgcsccHemdezccuaKRyzdwfkrZsaLBBpLKHVdwWKPEmEeJGexEciAzUJWDGvRvQirmuAxxLdGwBFObmuktagGAVvVMBdIHJpgcNjxWxvnxgXXPjuNqIsLjRsyMgjFtShcdtBbHrDXkQULmwbxvaoaTyPFWiLHJKQsVlYpCGzabIQhjNjsDvICxiDsYEQqQqkOGABDshgmMLsprSWafEFkDcTeOJtiRxOAsGDbLoyUUFKlLbstfmWRPlxvkKYHNHDWecQqnvQwnEpYcLOlwNjBjmyvpFtAeQgNCgfBodbEgImbZrhasofbZDJASZaKdxXLGXYptWrWoNYXZIYbpVmXSQJcOTXWoQAMsknjPrhtGlddWPXNLUJsxRRpiclhleDidtREbjhLWTZjtXygYgfauQLsQLnBhRENYteEHWaBeEsrDaQnOzKisdlhVrFXUxAMfLGfoZtaiYgmDdzwPnYqLjRCEOXAIczukzMuxauNASRhRiRDNjGEhsXmFguZmEwYucrxaAeNgTRtGxbWsSXhsujICEVfzLTZZbsCWsbacuVfcUMXBspjiyiuxVVXnlBzQEhnaVgTPnwuAbzJMbyyWYMKwhAMZJCwBKlAhMwPYyycwlPpAFsufajEsxDInaDoWPUtFbfDjmiDuyXWhlTLtcNoagDibeFFZowyktiXBNTCifTfVrQuJvkMfWrYMUehjFWwphkLqFUymGcpTgJhhMmOYFUqaLcTIXHSXqIciAeQithAObGOeUqsbYTtUmWYSeiFQafZqiEeGKswJuPYxZzMdQsRCqJBbEsTbGABzkvJnAsedAiDUVOeRXpduXFeqBpyITLLBvdihwCExqTdWHnJJRmzpItPInbMhxbHVvXYxbaNcxhDqtEjARDbDcHtaNsHcGiUKeoGTooFOjoNghsHJmcBXWAbjMIFZAONMBFTjBnvrSZQgGOTmogcgzrdcvOhQySrXeCSIhUeorYddzDAEgykXzsFoJAzBhOqAHCiUOnvMHkGGLLySoxJJNgHOCUfaDYlsvbdjxXOMWepbaKElMFBbBdcVcpvMGIQQZYKkKkAnazHQHfaPdPTbNLXEQmfQFiJFNivtHrFlQgMxqgTmLqSHeRSGhIgdnbYwRfsqADguNOOmmbZhXzLWJMeaBxTRnbaWRWmaTzxmxewdfuLdrqKrbiekTmQYokJAppbBsWDdNRebQpFQDawJEQdRARDlsudRIPeoZOkvzwPyVAuVXkyVZvPcfbbCSMYObocYLQeiCqsuOHlGxhbrKMVnGqUKNonexHGpIGjOkujYPlkxMxJwgVeOLFQqKxbhyErSeSYakMsBZjVbEKbYWZxxnqFeQAcimDSMEOFQjqczbzUCapDuiFXXJzupDEpNUGpJAstKEEffUdYFBBnloynowiAMNbDevfbIlsQEzBkFjLWAxTaaMsvDHZrdDpHRUByAXYitkVgKUuNLlMpYIDuKfxSzbCKdKOthRcyeJwfIwyINBjLoevWxLvNXixoiRRfRikDqVcPvqAZUhKCGDJRWczdgBqqiZKGHLwryYbyfKvvyVVBfpNOaMadqpEoFBeuqjJwAvKigsEOkYgjqblrkcXMUqhgoQwCsIfNXzEXhcKJDTWHOEptQJsStjSvxAImXXathabmSoDLhKIlRBFmGMZjSKvAlzpGAfbntpHHqhDgSGPPOnPRMOWmBeosFKzfjfFsazUgHRqBNwWFNCHzjfhvJyKpLvEXZVJYFCzfEtdoNIzEtDGGqDFHDjmedAEHGruIDleYgescwmCbgIHSOfFMyOOsslVnYIwSXFLVonwryRAbeIbMlNUdUxcvANKbuOWZbPeZlGyJELNyqGNOMclJkkzoRHuaiOwaoQdoIYyxJOroUvUNhMeWdODdfUGIOyRmuHWvfiufNdOFDfMXOmTRZZlObBzqrdBxIqnUuqtelVpPIGknHROFMbazMnfQnKflcPyXSuKKDluZNkZVgFQqdtrGPgQgDehjwWcOdAAueJjUTSEHoNHDXdACLeVBgwRSrgQaYEnwEXBOjxkDINdwNuobWWDbgHaNUCQSPYrWWIIRYNglTfVYTldZzdXFeogNdTAkqiHAxbSGGZydsDKPJpmgUIKugamHKkJTgctAVDwqPtLFzIMPNmiCgmZSxwcqmHSKyRUQZvvDafHnvAowdwGojcWosAwmcLuFTXDzsFHpRhNRClBxyVTjUvNWlHFZMizmDZrsEPwWfoBnsKiMTBJhzPRCpSlGaNTJbODRgPvozVbjwCqmtGakgeOZnvGHgqvvGSupKPwyYurEIwcYumobvCjZTePQcCvzNIGDgVmczlZtEyxqXGvetMNAVvsouQWjJkrikRhHhjijmyLvVprsIJdBOeSMgIaeSrnwUKhxnHgIqqTofityMZAiMJVqXoPWFPZqwNozvxWohKLjfXyMvQZIJGsyraygZsynvhxYfrlSFHCkraNfOqEuYXWQwfsfWMagKYFmuvGizjDXDkgtQKqKGpymHzMrPOOiRzQcHRsdSFGjTFNvKtUnUlrClOaFWqUthrvbxREEcboxfdWBROgLxmGZOmjhtvSXHXmVNkyvdQqhlyqjPvPHFvXxnwJzcwlvXnYqiNCSkoOeIysONeOkdvyjEfVIqPUfajVMQTUJjEBSCKhTLeVgvPtJUlGUPojJSiOckqJBGOsYSIGvbyLfDRLnPRMjBhpHuKEizpBzAaNLFbFWRGHprsiQqwmVHyHtIGyGQCDNTVyNvoUTcftOtjGTOSyVkawDUKcbIMmNlLfyIqWzJvqpmRicrhEIfBJfmjHeQngosZXbvJMVHVdANXpncLCPcIplfVvnMUmnqhpDlsItHPOwulFSMWXcgAhVHLQSFEPulfTKrWdyJkmwaiwJxWlvnhaMxGnIejGrVpcTlzCxgNCvVTEwVfgwGMsswbHtsuiFlLzDzGrUbfIpECqtUWGUiiYzlAkzcileuzMTaWlzehCERFUrYSDXnxKSQLYZdgubZgmvhwzrYtlPttWorBEnrzUHdJFdRoLBaZZfTMPMtAGCxTVugmymMKgIaJeDfCxLuJUkSBLxVvFpKRJBDdlvCloBLEYRIgMstrgGociHTjEvYamMAtxeFgcKnklcdgzbEFOyjKdormeTOZRyTFqGRhicZnGuQVgEtqbMmBUTIkwcBcqgHQMbyVdaadJxUtKNtTCoUVqDDUFJXfpSweSuiPLGdyESnqacAkNBjUwoPlQxbQBAqlWvjurGLQvCkmCkwvouNtdeHCTousKKbltbqIFUnKutMzYEpFIqZWBMayBkNMtmjFocuEnwqNSYmdQWJikkVNWgGOYNytYqwdEzindrcmswNTsJlajNvVgPCGeTxrRrNvNLJiZAbjefXFtUPuBuwqqroyrqhlrTjWkVwYacTmQsHAvqGHjAyQrBGIwobnotCDjcRhVENMoBngFeeZufWTZRHTsPjSglBFMheAzeyZxwQTKXSHSTSjJnHToTIqbuvaqmJCutsYNhjRcgGhjWvymVHBYNROdYyKxcbejNrcdIaRLGTBDJanaaPtUfrASZYqYbOyeytnNtIaImxtTVMdFoxLIvQcuiKEGGjmDYRqwyheaGtpGmVGFVEsEzLPbYystQbpcwOMqKGHjUuidbjnHarrwYLoPAPUcGIQKIaJZGZOjuFRiOUdJfFdyoCaabDmTZzZnSaQgjDWgjGFOuPzeHvVOXQeqwDqfXNUBzYJskFHgzRVHfrcKzMBYkOeiOljujjVqpgEyWXKIgnXtZfpwVNvfwzQBWvWLhCJRljtpmatDIeMwEOJVfSXEuPgmsExrtHRcwdaTeAHtKUSvUaDYYxySiDlbzRnNIjjpNuWodDjJmTYwlkjJrKOnuXMonAPFmBRrOqjhfPVzuvflFIpcAApXbntIdRiaAsOhpwobuSuoIldCQNHEklnCOKFBzmTojmotNaYtPKtmuPgIkXzmaBzUaovScZcwlZEryRNygRfgsYvVWZrioLqnfBaMFxDKoCfpAIwOtwTuZYtUVIEBxoRuWpLwpmTmrYYIvQQCILtqeTlpanhsWEiGHxrfniKafdOTFLnTlFMxONZlhGPDdAeKwxlRhBpPKknUFlRRLLkRMtusqVfjOLbVNCcqiyZWZSsuYAzsUughwkIroqyAveqphiCSuuubvCTBzlyfxgxBRvaXIHaVqMAESLTxkPCmKMGNoepdYQDlzanGAJjlfWMcDzfICCrSTrOSSyWPTmAGAJSLFDABWtKmBiJKXiGltvJRFyyQuitExzmaWcvpfQwvVvSELSHDnRwBfaSvicCwBEhAKPpeBgtyaDMUdxZjjFysxZUTQvGNOZuEeJSNfJEmxDTsSfvCmXfghCORShnEOpimoHNSvRnEllkMuLBxtUZlzWdylMMLgKrGnIrJkLicTlKfOTubJAnxisvxGbmGlsjRmbkcxRzCQEpvfFljksRdFJuHqCkuzpLaBfSrqSwDOXwdvPBeHGMRiBVFHrLmpSqlULUOgkEmscIKfPtLMmHfIfDiCpZQNYnqLbQRhLlMTmWfYBHLXqpOBpxhpFhKjRLhGHvkRWJoJInFITBrCynVPjDLxfOcXXByiYeGphbejizSsLEkywWZqmEeQgVmGdWGlXPrLuGSqMaFNWgfvRNsDVqtjhijUisjnQOpUSmQvNQmjSQwMHouGffESBomEowSkTvhmWtrURzvOQZEBdGilnTIBCZNDVRZSniJZfkmUCCWtqEKSHsSzmFLPSDXrMvNevsEcvZWyvZAWWObqZWNnoFRthpFaUEZYxvVxNxQUYudhNLFWAyJfrYHgfLKgFXuiIgAOYaKmFtvletShxGUAJEgWenNvXnzSJotXwvJnOwdxEsRWcmObwwQKCuhNRTiifbdOSeHrBgFcSCIxrhBdBNWVBrKfJWqiGJGqIdGyrzoKdYoURiqlHbpLuxHpxlzZVGALzJkOkuslvWBcfBOdWPFnCCTHIyYiBeNAEBWcFZHHUglUsDDceduvEAVtEZDDnRwFgjYhPWGnIKwgzMPnpsCpwqUYCsGMjnbofibsgIFIRimfFSWLieCrMfwGRYIHcmFyEaRdViujVucKBlJSdZhzWdRzbnXeJvnHnFfDErNeYIwIrUTKDYWngyonSEvgzZqTOVEBXTmqwGEdIdhaNmUHljoqCKTRARwTEXdniSOoEfUubeIIpdezpHRoyUtMTpJeGCbiPRPGxjdBNbwpzTpwfbGdTKUZrCDyJsJNAYGhvEGTUuyXMqwwGRudlIDSfOARnghWAFIiIzejGgidalwEeYmDPTBLIEyLzFjlLzkXlvJjHKQOGWhicapzoTMLllLSXDOgZBYgFsakIzaQRlqnOKALlEUWmwOKYnzeMuhMOFmfYWtympesIhHrpeEfLDkuppbWEgWOFdjwhMZKZkTLoBkythaTljZRGCimHilSMivdoPOhYKrsMLafksMoOVWloaVDnhxHQGFcKuwgJhThsINBuETqIVOUGmNgcMVZibShcxBbXlEOZtohAOwLtZdcHKCmZElksTYUrrucRGtdblmKciVnlZzBRaYwmTbLNQodWvEuIwGEyLJZaYRRKjLgiKIKthFEnMLUPkgFOaVpoNzwJNMqCKeluKWqshOglCJaPPeYAlpplFheiyPRxMjUWrNerOzLkgxDmfEexwfTthXSllfrMzfutIzPdXzGbDLAhPYztsTuHqRAwmXpFOMLCdsQHyuhWeFrmHuuCdXIZPwYZELVBwePwaNULAhcYUhprIeDeZxnklpeUyerYhquOOrmoEABVDmzRqAncyRHbfwXDbsoRrsZKSsjGZhdJGBPsRSrLjiskjyGVWrSPNzpBGFEpHPByFNzElDbGifpVZgmXoiQnoXffnueqMKkfPJghQPcANuibBKZazRphjKBiYIvWfCeWHaEUArVchseqWmVTefdcEAoZOrgDEtsdgiUesEKFRaMZmVAsgcoXqXLJdnQmSPpgtyvBtpYjwBtWvZhGQSCibnHIivCJJflAroccNtEvQuNMsPNArOgbXedXJWRjaNRBICjnMKjcPrSnnxBGuGfHafKcXnQGWLawMJphoXYALxLoEujrIfGMyjwJiDUyrdAeiaUbOWeuOpPGLsirIdHyiPMztqVdXAiddKILPpBbCwVFRfTkNgJeNMImeXRhzhlPXRptlSupxXfYYdUePXnuNOYQOVCPhiDGbtsTuxLMecwVYJacSqrxemUhqpxmQKlQqfvjfrZEQvXBPDBpxZJsWrVneAnXJyNYdNeAhApBcFSeKrjQBrHZmXwFHjYpigbkZMNySZJjOSqmKchJDStxpzHnIsxxRJRwLpHYlpfEmUpSPTWlDvmTiALnIEwFTvBmCvcNoxSGStaKFkYWNkadkSVzjbHFWhuWQUsrwnStxVWuHtROrbkxEDFGEznEmLiQvcNIITqaitbSQokQcSkLzWOSEWUeqahHAKlpnbmKZTNBSKXdaZXKQiOyqCTubkTqJSGjpmHqPtGvrPqrAFttSlmgyTeaOshLNeKDECpvmHLiCjcpLbPKynnkJhMXUQusRtxIRffTAOMRBxEMFuBCbBoPKguuthmqHJVLmjKTMACShEEZUPBiIzUiTSJDNEfXUKtuNsEoQyBmzhWLZJSoaexGRgcFUAhUtHaZFjHksDiNTcTaXaiXRDWDrUIwgxcLmCthsiaNGihvlUMpxpLVPAeHovLHmIYlNGFMfIVLURqaufrfqXcdSsjQlxpQfKZDEcrkVaPzRoOQTmAPpvUSAeyjopyvWWxufEHikhWCXbtaGDpuOtsZteSbjQjkNvsoEfdXKOBVWDlkAyiBvYeBLDgyCADALqUIjUytlxoVpFFpkcACDumQElCrLnGoakEkoxxLEvcynmAWlegKHzXxsEnmrGcWmvLmaCouobfrCtpvrrJQJgKReaJJoVZfggVhWkRcXsOEUJaiAOSarngTgsNVAQDgwZoyvKFtEonMbZgnSCTofxbqWTExAnMgTrgoHseVlcwpDJfySHYAsgeECkkVOZhwqiGpougyKeimKRmsgAUkKTgDigNQWGKyyQTttAOrxXkWzpNzeQUdqoOXFsFwCtWrKQujINdnYFufyWKdpzWxUhsmSgGryRAOCGXiVgOhqWnFyJXVdFJNSXVKbQFatEiMTKBckBHljYkjHWJZZxDEgHYXXBOKbPLHtvasEhZWyiNsTLtRGbgLDHDzqbUUwwJcuRqanWNvjkNORaQhqGzkKLstcQBEmKsGcjbIXOeSDEsyOGMKTabWskNbfIsxgzxDRCVCrlVDMcgDjzqQSbjYRUunOSqXytNYGYMbgZelctofbMpuwseiqPHyxMlSuUjTEbnzzoacbAUOZUEMzNddWLOYXhicbtFualNryScygkrSpnwCTaFuCpqicsOODIMuptwFgnSIzczZrZZjkINgGRPMrzzvDibsbjERHLwZHnlRdumFQckAWddqVpFUFlYZIGgYfGKDcIqjtTXcPScfoDbvbkVmYaatbmdIIvTatFDMnXojwaWjpIxUxDSEoYbEkUDrRRWYlzRanHZNNvLNNVBCwZnQVWojrBqOtihuogdJBvWQkENSAwqESYgVwluxQdDQwPpckUyyljhNPNXFHAnraNSWswAuWksUgevGyXHFqrUgoVVNKHMkLFdHIoWqzjNWDbCZXQyFIjOeSfdbkDXzyChpgrevarnQiWMIgNVyHMtZcBVxUuAtDAmcaMFBvXgNxGADuCZjHylytPNiMeuHtdfbwgqYrOFbyeKXjjokeBvokiJlVZSXunzOqfUyvfKwWsPaaUPIpNxMJRAeAbUPdVddXSmBywgyTPnfaFvECAUiHCBTlnzFeYmiIrDtGoSjswTmTDpjblqqbnFoZUOCBLUlrljXavLiWcWufSrLCHKeIboVKUWpEjKzcuuHJqnoRheWVmyfjVWegyoXMVagxQzolcignEiLNggpJkiKRxQULjHvGjrolgIdwPUaIEWTNdDTqqBjdZUVTmeTlUHpMTQktNLPjAdgLWvvqkTyMIunEnGOKbRMOHRtIGZFoyZXxAqSZVKVHztEHgpMSySlpEABrKkzYGwPRaAirWBLuBZzajkqrgTXCmAABHHPKhPFNQmSHGOZJiTmQKWobJYrntQJTuFrUOelVHDtCPLPJTEuiOCAnxuOkShjdlVSfOgMcwbzgCJhWlOHegTZUfDGVfZeZKEHIcCIGAOmGBwscfLxOZyKkXDLjQujkuEqesTUcShIaNksjeOuLRTIwiCSMkfejCcuPPbvZxITfdrDkPknATVvtyqzwUuIjsrJbUzRSYIVwIKabmJdtFXBdClaTjlHfLFqfzvdHrfesCZVAwCwBHySFSQEpToPnjHRAhBToloOadjjDYGzazkahXxySDwIkPEXofxOcwRqmlwiQcxENvaKtkOmbRLokvezfPoLyyxpMvFvUHgmUANWIKTAYvnoJREIMHGhItRIVOhUnFEssNZHeiSmYDIipryhokiFetfISVuspKcppOeEyAeDYrKuybHykBGdwEepLRvEHaUQIZVWwiBrNtDOurMqirwGxmjxNqhwXeMEugCpJqUTuulRuIOGyOXodrqvHDeMoxvBGGoWWFrgptSXaSXRkNbZHujRXbHrOcaXfYnpBLHerzVGmaciYRrNuYsizPhkUIlopMniDtSArDcVhWdsExaMMpoLIBYZVsrROddMKQTZVzpxeYsJSRCqnQDwBWOMAhZPQwzNgHyRKvtblOHsCNZfUEOxalieZyWStonmPhCjxvqXGJsEbpUTmhgnEFBEQeBkITZmJgfhpPOPDqTkITcPEqclptFlgcUoaPPAncLcJXqlvrRfmHsGSemZDTyArSmCRTqcisJDlCGYBDMUpeUJfYNkxTzXGsxqMsUxcovXUpurFhLudBvcBiBISRPQknhOYomZkNGTQwPrIArRKqdyNlmeJZekHBoefnfthxvbfdnurDdtTiJwkCVYBwrlnKVaVZqSUcSUsjLJwydteKjDnbRpoUDqstDXURfifKnOVDMDMLmfDSUeIgFhpJtoaFiXSmlbNEZkwgeMSZVOsdiDWQbRlxToszUExgarGZyVMtEMbWNEveqxtfXpdajAKAnHmRWjfUgCrHeYTbbpUGdIkuGagsmuxAwqxvQsLcGnONyWnOkLTSzeUCWSbSQlODzKaQTgcfHeztGLlChJGSbVRghwuiOKxFwskRemeHjnuhhKZZWBDjuYzOujdnnaJatcVzKkpEIaEHjGozWlevjTgelaNHSkLikvFSGeTvrZzYrqybUnLWpDVPXZYGWqNrVThvPrxplukzSCFEpHJQTxkPCeeKKrqWeoUpmiglrXutmVZHqetntlHEqCzioSJzxClfacwUYkWziEuGWNfBsQnVGnjxcMlasxBAaoqfpCHCMFfmEsGKCEOcLdHcdxNPsYbbWVuiyUarDFJNZAdsrRrYHZXNvRLEhxUNZZqldevHlIguLGXOymoRyRDspyxzjuCSutoBDGUUcdxlLPgorcNrzuSKjzyXXoUjjoTLdIYCyaDsrAIXUKiyRcRPvOeWaMYDrpuGhbzEFcoNrUhXmOuOUmRIXupgJasfNJVkvDhsgvESuCTrXDrYUbaShOgZmNwIuqiBcmYiwkmFPkpCIzsPetoqWBmxcYSBiCwJkXTkZywkblhhPpwACDUqtmWMSpmtLTEpJiBKYwfrNgtogTZxdOpbCFIkdMAJUgoeDkiobYhhWuTEhxZohVGWClLfJYqAqczvtrvhMkiXAjgAMppInHiOrSnSDxwOWTwpBUJDkVwrmAvfqnqIXInFpqvXrrDoTcCfZzMjSHWuxeDaiEirphwYnulGFdBBBEvAUdQdkVIVkaQcQoLIbsAHmJkqHpqhoJlEncuuZRBlIcglfwSrGnEulEXlAZaVlMSSAwtBLfDgFBNohoDYzWcclHcNniMVwiNPxHTipmaTQDagfDELZKrbepcYVJagRwYNqmHgHSgxyILkoIXVBrXaafCcwOXRiAVCKGFolCbVCJCISjjIBcOZDjkJkTFWneDQyHIirqDkiGkjXxOtDagSorbnJGIXusOWzmSUnMrllYGQyrkVGSXnKhZLywxrVYjvWaQkFVRFVaKTEmdYpbeoIRDKninGksOrFozxywtpqFfIVeCRfCkgAVvBTamdwzQADprPqprrNMBwEgdJlaXvTwBHAcoPRzYTYzzJvJDtYcaNOYGGQMbFwrEldOPdGYNoqfBfDLpwgnotIRLmDToslbneZBRexlzuIsQbPCmrMhwHATNzhMbZLkyHKNpaHBQULhLiPWfSxWtHQMRaqFChdBfvxJIOEIJTFwkHNPcHTqUuZToxtrGHSACxJbPxFETVuwPVkjUFtInwcVVrxqTPcROGynomHgIpzJGBjuqAJYogCNqZQJcfGNHNmipnUDqtLBWmQtHjoCvJvJFPfFDuOVZafTCqjdtThgcRfpHzXhzuvtnXOvQRVhxqCbObldoGMbNlcqfrEQHSCdLKHtNErwQCRDQQKaiDCNuinMPfIAWSNSDffUtwvJerWfcOqoRvlHkmaPvJHPyKFPQGDuRKcfRNWlCUdpxyiZxITTNVbEPloCWpcOcyPafABaOpfEWQfApsbrzMrwZVGxkwaqFRpbcdLzLviAKIkAzqYqSJrHpVFijCYDhqKWnmsZKPseXjVHHAbKsGPUIXGlbhuisVnSrbzzcGPPUxNqtHJOLXTOdtSKOBwlpJSRGtfrSOOJfDWCoCShrHZyJAFFwRAQChHwflutIwGQDKsZKPjgiTGNEuIDCKhQpmpKxpUIuSvHBrdseAwlINVwilzfiJDHMJJJvrHrNRiNFMWVGcYYgmKixIsjETMZLyDVdoIClzIJNKmLqWYeynyBsXaArZJkYWNNdEtyIcGTReUIDKPWDnKtelBrHrpTGsWGajNocrEBeesfdaSzBXgwlRWCoTMSKWhpkGDemXPiswFrecdXkEDnJeWIrYDEVSKRBcdFViKCqNJKJLmZBesLMsFIpGukyvzAAPniksYJmBxziLRQDCCIttdDlmHBVoOwmFVurgzhjkeyaPNWypXyyjLSOhgpNmMjmenzOYNWRYQOJLwGLZVRrvNXqoWUaBlUjnTHKBHRTiUYjyTSpleAoWwHTEmFJLtZuueZVkqbgMfALNLVWTYyKPijLcademiebmicycpDeGZzCffBzZyrdhaLDuQbGCSzgLXhOeIzLwxLYPGibzVugjXOglGSqpGBFppCYjBkFGyGWtuVdMeaZCMFjMcsWzgkrXCaAtxxTDYiCOvpBGzvSdmWjSPOzszYCmCovzLEnTlxlKlsUdhWeLDPPYvGqVQbjORmbsDhqsjOauGkzjIDmKeVNykqcySCnNNhpQQnVvqbNhprILtGgfUurLVIMErHewqTJBeSQyHsdbODdQkqlSUzjvcGSWkRYWYdiUIywkZuoVvTotNCtvQWAhnfTSDFSmNRoknxfAZrppHUveacqtIiQobcXISBWzYNroLbGTYzqNyoioWwgPBSpZEwyDxjYUowSzFtwyFpHfcIelaDUmJSmpUncwwQeFOxoSKdDCmYovDnPmHOZuEniAhYMTphouKAcuaIkeoGMxmesrXBOQUJfciFPWCGbzriVqfFDewsSdUgWCMpLlwDVRUhCcmgXGCdSHxAlKXbUTRFGioaCfuoYtkenMTXDNxCUWLfKayAVxwWUgUMDbOpVKxCYBTVXKMHqEyCkmpwWtOfaYFoLpUyPPOdaQmXCNEdWuWBTbYdpuEmYnhnIDEcEURCsoQvlybaoTpGsKtJwGvCpYDJelFjMjsQmKkvqPzNaNUvudVUJFXiAzwpJJpRdNXhPbgEivjTTiKhflBAFefaKGHmbPSDSHBMdMaORBYnPEnegkCpQLldDMtkimKSLAyAPiqCPWNggRqEcnCZUGpeRBwQbVqfCWIqOqaMOEQJnhhJcPWfDozBnjnfYrjPrYqhefUvZgbBwKqdzYspjTeTMUkUgGrDCrvZwHjrdQTuYSeSByTgcauVsTiVBvmuGeGNnlWtxIjYsKtLPybkrkxEkitAjGEiMCSDHeYJDPyDGcdGHMveLAEVUzgQWeevPLDBJWTfGyPaKOqaDPboKtMRrRqdijfayNeFxXynqRPSFDzUUQUTQxdIEmltsnuDFrdqiIdJjdbxfrPpLgDtGZZywGQdyJnCHatRDVJVMjTSssbSiSkPCRuUCYEIWEJfMYLsUzpSNKwcnBigKkrwDHYGDXHrFjawAvoTVQgSbZAmaXDOiTzGEdFsZCZzVevFfyEBHBbfTzRUtUocUGfimrvPdWvTeqWcUgUZmZwFxbOmkgcULFAqcDKVrkWQHztoSCkCnXwKoSYWSgBLcXmlLhpgKTcwiTZtbVFzuYmsIfBLMrEjkJxmfUBYqyAkNxLGOVPVoYKFqzommeTJnNnjlckOEgJQKwuoInZVDOKyUbWBtXoqscTtjFbVqFbyGVKeTcgGNqCxQLDPoPCScVoDrbnWZOSGkSYvbdcXwwrtyLTAxZxxJSmLbxwhWhrShfioaTqZqoZrtSmLaMsPtAPpxCZfbSVtatcfDpcaMYsoZRJPQAMkllzdDPATCVYvciTBOQluOblhmPcrCnEUeFBEamPMPIluUsqVmpBkTKsPxTMBYSnKaolSZCvVYpyBJuuTprkgvNDESmBdwKzYyAEoQtRldfjdRrOjHhsUjIaPePtiZHXxydDKYWffVHNFViqlyEWdIxoSKIFYpPeBAgtrzUjAKfyEmlDOrWsyzvPyyesGKugzDLlIVxnQpkAjPCKZFWFAoSFImcmACKJCqlFCjNeDTtEBhUenTKcsLhjXmMOdhIDCMHpJkmbuOQehuqdUpCngNFRmODhrquRbhwOwjDfmYZEVaOeWVCWLsySEsaWYPfgQfDBKklKqoFSAGnJUKeDJqzQMtxWADmamqWYrvjdiBYfsZLsxqEjAohgNAYmJyfPNGjwFNKaRKEIrBlfwxLAcYInJZKZNFVwCqSORStUjckGntUlIUJiICHCqIkYOJAGxCIVZtXxvsPssLASvlrXQwrYSoyjQWlyrDLBjsDgczFhZfpniiYIuaYUGuInUoTvmKlSJHHrnpHnLoEcBwLEXEOjmEsNcmPCuOAZWsNegkNtKlpQPpKQNrOpZRHZSeZMyJFxVWoYYCTeSXsFjtbbLFXCLZMMszubpQxnBsBIuWMdyTxYJLekiSfCQdMggifdBUBaEBjhvizizjPehXvhixzIaXUyIDoJaGDVIcQvByfbZkHieDlsuvDvqzktRhFxuidSeCMaqCfBQotdatsaHPIjZATBInYWQWrPbXOAPWdRSucCQbLbOfllELFDbrBmhagHGpkmbtQcApRdJwaOGXuzQWRXCKfuaeMwTGYSjqqkFbIUtAmOKUEvagckLptckrFlosExpbBQTDYJlHuLEjFdfSXVcyfyGQCiFOzfCduchVzHYCaSUIYjTsWwabNLfuMaBgWqvNobdfUlopgZhLxAmDaFUIkkAoSSWYlvRmBsEqdlqPFWWAcCTroZiCOzVrYBzolLXdTARNECKQiOhVPIUKsyGWTOiOmDTNtXelmhEQVmFTiNzbaYHJJKhHJkSXlxMjSaUbttTBpgojsEzCIaNzZRpGBUcSgdPMslxFEbRNyfFquLnMkWIVgvqnnxwjtYqMBervSJgEgQwRMZiinQBPtWbNewhzYRyHSoywWWukGsyEllvmSbkGnRhqLoJxicLkKXNwkvAmbHLXEHYLQwjfOsaVZOjSdFhbsfFQwvGGbXUJWiluTWxkrIkObXZreHXVnOueRKjVJFTGhQDvpykapidXJNLMByHbhzuohVBvwBzIbGQCyeBAVrJWhQmvZfTzwniyKVLnLYQbcWnMqNhYOhHNYPyyibWdQjZrgnMUzzcRavHhwqeJoLosDKQGwIfxnaczztKHPKwcoRVNCyTdzLNrachIRbuMWItjtxVgOUtFscLSQvlIURGrlBxzjcGERCGuwDjKsmFgDLlhHldLsHujkRQgKaDrVKFUEEYykUpBqfSKJuOWmSgxajbmMraMtOKINzEjrPkISyGkqzTsGBERRyzfBHNAWXhhuJBnWASLfdBjSytvNFJZzOSLorkpMnBHIjMWploSjZwxRhDqBGBFLVKCLXBojcubajHwyBrFIQEReORHHEXthzPQmRiCKYGmHLnIfDdnfnQpBYHReIkUbQEbwoCaLdpmyaPWWYpMYVxpSDebaEaqgleKJWaxDvGycMHHrfMcQLLQKsLIoFsKiCfreWnwwDFbQcrWgQeqRYWlpPLVLdOYEPnnVWVrMrUddHPTUAxHRnposgUcqYpKDQkAIvmJpAlXCauilwvvcZRtMeoyxWCPPbDOJYmntdBqoUAoXqTPLOtqvIjRogYwEjsxNOHvpyARNnRyZxGPLkMFumKLJdYWSZtmiWsXGDKpgXHgNRskQOZElBfBfnYSKCbzWjhakTDsWqlaGGVOTcZERDrwItGOxDqLKQTMthxYvhNPVlVBbkPZLDtsWhWMRWqLrCEkALwnStenRSFCtnCIFErUfmXozJTgplKAilxNGqwUPLgCYyJpZSwncBrXrOXKQpkRqEvFkiqCWcYMPWwNOflyORzvaMlfAiuPkIPEzuuhvSmfYqoktRmhvcsqTxKnerPNtOwgcTLAflbvlwRlahEpczyCJblKEcvRMgBTUoSFyZIKaylhCalIOzrgzfUtOfukRyVGsdSnJyYIgsLhMEEPTbtRNwcnrCDnZLSUSDHGecpqvVbrCcFwSXvEvJLVMfNEiemZbAHOVrmHPXClSdtkPaAsMnCzglqXhRfXjvTZvixmYoQneuHPMgJtWbMHRtgNowUomUxZaYYduEiwnCEkYiizAUJenZkfxMLpMXRUBjBfvyFbVpaXXKIshUFee</t>
+  </si>
+  <si>
+    <t>ZYFFJPhEyBoppZlbSaVLmwnPefbkdAnNznmWAINWdlbjUaViTnyomkvgtVQoBNFwcqIzAeesholtgDUWAiwtXfZkyoqfyYZunsBiELmcjzWFZZmNpwBEARDaSjgVQZdhweWVrBQCyMJgasKJGbQfvbiGzCiVaTJBwpbXVBFDBACgYzCgOPumnDSTzSMppUdlnOZGeFrNpetpuWJrsriwWZGHNkyJEvWhRVPMYCykVSuWduNxJHbbxBwmiVsArHYKQOLrepgJKuCdZftOBivTyrUHSrLrOvLRkAuFBlgNSeDMJvjJnnHedgjEzWAbwVkPjMJovfPHYKsSeMWMMKazzOuvZJZVQyGDloGVlxfjtqWdEPkZkoHnqLDKOtNrNaykkofunXQPScrmVicQgXfRDxdqZYHHyGOugCmBPMYQsXypwafQsQAtOQDJqaZsLkhSxCnofgmOLwUDYXNiXMnyLImfJwrdgjgZBmrwZMKjpCZunciklMxeVlAlBNPviyMEpGLAPXqebqiOjfinRhRTFSHvvfOUVqyQBJSEEOVONhJGhCjezFnLPeqzMAgYjHKORieBhZaQHOrUEMSNQgduShXatpSxfusgBDiquIpRqVEWiyntQvDwKJiOWrkjkhmMEZErRaElRvwtxnTyusPXhdqbSFwaKxWjdURzDRgFnrVUOehEHBBECaRwMwqnwUWdIGHtiyUugbuPlSguKXqebKdSgqmqaThVNUnavnizDZpYzoYzofFGJWDqXAKIbVpAkqkxLLWbMCcnPLVggfVInjLNaSkrigwOsEwgKJWBhcBnGTzcREmaYOZkOZPbUPhhpjGwNuKIFGMRIxqOlaSCZeNCHOtzLNXpVgMbLBaTXCgdpuEHpOcTxWIWdXGUOqCBwWdcxShbQwwtoMMzDCFFicjOZSmUXSLSsndsamzsMxxrEFwwiAzlSGTUvUnVyvbcsMEsCmFXGHjvHODxkFMxEZNTYQXmoQBBslDeiEUMJBRiLXqWICkvLpURqSAhtpQYgDmaLJbjVohGRCUCeZwdBwekmdajaxDlBaxAwCJTAeAmNSAzerFBccLqPjAwefydQYjvxQxqKVdrcVcSaEnmbzpUBoItrqveQniJeoEcnMOflywzHJwERJHuiOyfnHBBXqxBXodqsohNojVoZBLjQrVwrdQzEkWjgNNSUvhVRmHHelAwLZXYpvBQXiswTsiWhliRcWnCVqLzwNyTGYoXRFWUUYkYWTaKUlBkaXwwkEJwekmVAfQlAGxUevEpMyPkaggMhoHgISGAJzzPpAucCMvPtNoDfsLtEaQgfeWQmyTkCVNtwLFhxTpqvsPdwlnpyWrrBFLYENivurXINzfwJXgpqpxSLhmziemTybkVGBQArXRAENQRQXQOAsuoZFVDejwSMCYkQltEJruktewWEpAdHwITuBnhywtIXVzIeajkcRUgeFkqFXOvmncGeGoRkPYtUJaQAUqtjpPoOMrLqLNMymiSRAtfLMJAFIKxGjWKBoKgqTrgJELDJAwRSzyaOuIOEDkjBVwfZuLsvKCxDRRDAOBSfDuLClEcTDvpsvhoepoTTOmNZqlpJsvtEGPOqYjCpDatxIKqjBCbMwTPfWSlKMDCCayLYONYxhZhgvliAHIuxHCcsiAHyRwFVPiqtivHpoKjotIUFpEKCQrouoPfNuMElCGawKTDPhXjLpnUvFxtUehIaNKEepeoimSUIhtfeceaEPtbBBHdSXFzPciiZTASxCsIiYEpHwFEYiEGyoqleTzwTkITCgKxwovcDJCGEtDLWuYzeNauyOlMcWyDlvDbMTPnIQBJDnbMyuALzUunnVDWrsRYUAznhorOrgoRJTMdohZVyOELCtEpRgohAozIpgKTKvozXrEZDfSkXKWYyniHVcIyFadFXJIJYeaWGYpBzKFqXICcKDNvbpbxSYLAvGMifMtTfGPghrmLhoppumhAOhFMrrNjPBKdxMRRTqTvFpVOoGWitxWRRJhZVQCRiJebzwZnPKpfANHGZIHJUTPSEMDGDAMzRopqOYYTQzTlfJJytcyArBQUrklkOAudjnETTaEfhGcLUYvjuyWfCBZxTFRXbUkRsrxZnqMMyzQvDhtWuMLbxPUaZxRCySmCEntQDrHNeSabBcRZuwmINXQdFjowFxjJcICoyusRDyUXDOnyAjodNjmszDDYnlQsrpGiNoZnItZhfzgKaBfILDDOsJOlefrbcsjlXyxJTGUYcdGdsCtVUSkaVcJiqkIgDgCnLjHykoAzkEEidrJGxmTDtNYraktBwcfvOQFkIzJsbpbJqztIpMmEjtVPsBbvQSVBJBoNzVVHMAFlKHXRnsGxLaoCWhBBMVeNzywUPyGbkhOqvcPvsYQZxYHLrbGNRVjbjZXinEequKhAtjIdhZZfzbzRbazMtADVBvvhOQQTXeXDPziwPXyDYPtKNcrEGMjpycRcGQDlDLQvIpRXcNYRZsSexJNoXVuXseuKdrTQEnnRkvOUImOUSQCQqJEkZHKYDKJTrUulMdlFTAItgCMUcdxdkuwdfgxCwTTeTeFbCGDIkeoEzmFkVBTVaKZptrgvIWCljIfjXdQiePrWoTwyotgcRglKGmbYTSSmAEcreEcFFnlcBRCCkqEtMHrLdzgfsXqKVedZrPmhOAcHtmxhPRtUwvTooEnbhoCWKFjyhePIojsXwMvndPTeUXJvIPsQPIHDjjQNHOiHtcBarzpkNByYdqDHMyOeOqSWVDiPjlbYqeGDVghkxPUkQDESpvLYhltnBqXtJooYHpdudrmaKcvVGTtkbvsKKxXavRnTOnzaVECtPjCaZjDwbLZqjQtTgKBSpgXAGpCcjKwcNriKgFKmUaMqtiqlOKXWYDKmejSnQaldsasiJPudRIcaXfwUpuZMeDLfBAgdhFQdhcuoZKWjZFZnJMVZbYHhWvpdufszPASLeBeArnSzrDvNkNqqBPSGGxMLGTMrsqAVwilzCRjFvbbVnKzbXZGnRycuYNniSPGKyUUZJyErJOHQtrxhaJEQehQESytWSdNOcoLdGjcUqXiWHHjRvCnMRegrIEWDcPjUQLcanQbizsWMTsErlbTkLFvvxBDgzUyTmHYfJOHBnwdjdJVpkayXZunZfVOMohQMfjmyqtjADoQjCcZrbXyPBhxJYkfWcZnbChRMMTqcROaSgNvHuFgSbXHktgQPrPCoBdGQgpDGWhbIHmSxlrEaazRLdQXyFumoMLdOeUFsdBufPxGtfrKONOwMnqGGmVJKUHLbBZcsZCCTHwFkSJIbQvKrhzPpOOZhQZygJDtZxMTrkJphaXufXdHyJEJzKVhZMrdSUZWYeduZrNVrOaPbdvlTzGFfQxBlXWgTzNvyffwEtpmbdPKqUpjKJHENYApVeOrPCBktdVbJmCKKhkLqqEPTJAbWNTlyclPUcmActGSvhBUdUehAropbfjPYCzsHinPpyjjnwsmcewXBloJkOuzjrLpBYHtXFlBsTXuRCzDKZCqrUuoGIjkVjOIVtjIdZjZQwhQlgqrQJtRbeIokkvUeCcJZSfYvxDCjICQibaqKbQUhpiXEPgwIIZUmgCrSRDcfaBKXPdItoAPOwwhoKaBMqaRBvPQSLDmWZdHpGziHIcgxMUespgjkNPjjTrBRGPMnJaQsoyztZLfuDAjkEyEqCNqRvyRNFhLGmqEKZZPMuQqQgzriErZrgLushRJSgBZzcJIYSjTOVjoyhhGXpLuPcemgzrQjQFGOwKnjNrbzdEAmewCBrQkZWoydqEKyLtjKMRjJlMJAWKxmFiNKdobvOZRhuUCuJEhKQhBcYalaQpYsduhmsuyrzAhiqkdfQclFROyatVZxgOuvMHgjGISxIkKGgAdnSiAZPqeABbyHfVgsCLCDcxkPFwWUXFpChVGnLtCpxBJnxkWlmHjfvixKzOxkMVJTmiruvKLjhMXmmHzqiSxPEHZGlrujkZisnaTojjwrGWETaruDODCGOOsHrVCjcYncYJsNUxlwHWhKWFUdEFRSnuSCQHRlNseQitPlshvFOYKZeNbeqOHvguRELTPbKVtpFlYKQBhQSkGfCnvmcNSgkmTslHGTWUQToQrejvfATPuDuBiyExWKpBKssyIRonbZZgYdyNKINNjdmFFhpSvGxaqALaiVeMTSiJLXerBWsXnIjbyukxnCLgkIbltVnjBnGSfMegwoHafqjmjSsmdTrAkuaeOMEGqsFvLIDYwtjEITzekqrRNcabhOwVspmBBGIabgQJKVpuQAvubYWORWNCTVPOIQfVVEIdcunokZBqGOcbzSYHhDAFraxZFNzPZmfDgMuMJQqSyfCoZrAVaxczTUaIAltoGyfOPNALGUIfivxtEWrAiyICCJBhRVhzCoCgkeAKWauAkWGjiBHVwBvrzMPCeOLmHWTXrshkuoHELDoxZZBnxrNIXTdNDSTjRbdynwrqhfjHTXtSmCTeJnZyBihsbODcfbTSoURnwxEYToKiaxytnkUCuHUbqSjqiYduuxzdKbctMQCQLkIANyUJUVycNCnymOZnGFtCjpqpYsqzxOdHNAhKEvQWJvJGYpgzoVbhMQNLaKnOrMMNyfIDspWZcaRpUMyLhXNgmSiVJGEUQPpTgMRaFtNydPSMQvpdrrTSPCauSXztIgxZDgaUVvYeGuibCGHKolKSRuRoVOJzcIxWTLmVivSqPKQDlvRqTfmJVQufoBluGGprtrEPLktmPugRNZjOPjWrtNMaFjCKdEVeoRSQfLHPvyGuxfGwiehILiogmcMpeGLYiejfIfJQHxYvDofaQdeFlFUxSnumlqHjiSzMiDTaplZuSSnBUFEnOOVnEAkPSJzqxeCPdCmTGddBHuUhDmvytOeYFaXRfkjkzBEpYBVEPlBrsYtBdVroKoQTMiZnTfZuOhjBFwNdKfTdCmaDqdsbClCzqdCalvVSaXqHqDXIjWojSeDkjmqHRhKXBJmZeLtWeIzTvuUFXoHhrIQppCqIfnNqVZMSbvuLTApXrpNdLhsFvSWjQSsqDSuCreDRvdjswGpZfJTwwLRxUhsMEHQOBpLFVFajVXFuExGdcZgfVbdScwvHRoaDdLDFvRHxwhsYGlrvSwjsvUSVsVqTetYzXtWRQLwvGPJTQEuYStqRbLJVghXbkSSWryNAzoPQfBXwAFdiMQNTraDGPpxpgcRCrsmpdkcdnZneDVszOxeOGxgyoCKfBkmYkIQiQcMnLJEMaGwtZFKWxVPMTfVZXgAaogijoOZhrZVadOgqIuLhswcCyPCnbGaKZihcpOvgiPcaBBJQdtHLOwNhzDcfYgXXfIXZJxGHRQMxYGTRPoGFTUpDmSLsafSemIHPOGuDJaPjopEPWUkkUdkoeytguQypcHAdzJcpILNiWfixvmjRjEmoqepIrARhDFfxaQOLbdJhayWmdEumuBxgNsMcvJSdMwxRKSHEtIkyLwYICeBkpxajMCcWfFtpCaeKpNoQWfRVUWVtclrkDEqXXGqpuPhVAtMIwvRGyVMjBifmIcUTqRkVyyoVqRLKRhDybJzfKpGLUdgHfLlpclheEwgvPFtNkcwqeaCTDBhWErDaPgjxWAeNQqHUqdBWFKVjkXBHoGSfuatbiMgSfWrFciLPXhBrhqJFRGQHWmdREtKLXfGUxkOehGgsmFRPjImLJMdUxFKZgXMAIQzmapVioxqGQaSjQNIsQymYgmrfcISTIkbAugFaVDEUTraLFPUPRjwlpKTQPWmLxijTRuWGQCpQNlxASJXZcsyZPcyQhspZJAGNyqTitWOFNxFCwcObteUFAbKazFqCYuchpoKNQZHjImtrHQMGybkLTETerYiDpCxZXqddqOhnZfkseZUnIEdDoxHCcoZMidWSftqsPkXnwIlQZfhfrNNkLFnEPJdYXxfgwuPtsiKuTrTQeqJMHNxISJSAcoKBmyGHZUYEtGCtwlUQmAyiAcQiAKeYGbXVrdqSCiXhqQbyxBlnYdPXhDaxBvYjmXzWABvNEalXwsRzSMwKhtZzYQBPAtWAYSagNgsSzhUQmymuVDQjgwfGgWPxFNhyWYuCilIQbZAakGqOZLzULiPqadcMUkvPoTBkaBWLKOpzhUrUnuJmNRQhLsBZUNXxgJeeAKLaGjFbxMLMDgpgeEsaoFjkuxAeqwLRXhtoBVtlUVfyxDhGJBKlTntFtUdkJXTPqWogSODSjpxZaUbuouXpOQtgaQSeAbrHimdehzJEzexjKkXdFaoBqPLSGtJmWjNuVfiDDfaWDeTePuqrwfrhTnInlEoqCYIKNCMBzqlamglYrvyvgFhSytUIOTfTtrKeVgVoPvzIExYCvXYiiNYEAnuzqYQLTjGWNTTcANMYNzTvnGRlhdCspofPbzdqBPbsiAkcpLwKwsXMnjdgsgWwFXvfuKCUEEXzYbEASLdswcinlrcJUEVJdCpOKojkJRjsHwIxQWNKrcvhFKzhRJiQDpBFUENPixAYbTEvsofnaBmaYAGJIDWLMLrkFVTVMVCODYpUoBXCwbDhqFbEVILHQztwIUJXzECmsQuPmvMyzCrmiZWepyQVWpVxZDBcYxwHgnkijVgsdcpPVRLOAuGrUeEUxXORWlimevbkgGMtacqaBjZGxnUgPLHEAIyINrHWsqBXBbiAkBzvMEOMrrYWlNVrIyWSkJPDPnYgeePKuEnrMztrXIuRQmvecgCYVllVCZUgKOJNIYgQlwHvvESdBoaNgrtijYnXeVgySElabtkkMzQXHgQrwgmZkNWloedFTqRMMytpITiBjVyZPXIbjrqEtblOmRtxCCnqvzyazXDRxnTpydVvJUCqTORJyqkFBlOWQmRwhxHrTmqtzrtlBHWyoxYdFwoAqWKAZrQBKIDiQUHVmpGZYiDpaEpVJmXCwplocqmuuxlyTNiUpSgyMgmJCyUtekxMILUOemWkMIPBJIFfXWUANqpweDyLSHYFPnXLucVcdYsrjhvnvkWqdUQJedsxfCsxUhyxwONFnTvmKWlWlfcExmZPhLymRhCWFbvUsIcfrBwjDIwSVjvdNCfcmFQtNYwuDWOuVrskeuNQsuAmXlZlYSnUaOCksZpJsLZqIjlaOtVlhjamPknwmaavwknGSTKybahkKdzFJnpzRDQdcfTLgnjogrRqOFykwKSKDawjlRusIekPcsiofLuoeKAugIfegHbvYUNguwHdghBwPgsVEPDwkCHsnEPyxVzJLffWzMZHvgyASWXiDiVsbLWQJbhpxXVGvwSEWntHnivpxGoRzjhjvoCIeWnWuxZogCijPWzSkeHQfYoZiQopnwVSCjZCUuFFbOzoSTeFMVFcCYwQEkyJLMBGdVZnlipEohjkBEtlRupIUGHJdVsffKBxtXyGbZaukkfksKbIFDATMMLgMsMXHgsmIOilNXZmZdygTfUIOmIlRbxralJLqkeNfysqOtYmvWvZpFNkjGumkvSrbFKYPasFdYUbsPDVxYxxgdxLLJlretJdhmgPXSZzWPlVMYJfkpYNCbvQAtkvXwOMmdguOshLWKmUkBqvOyeujyvqXNnSVOLJkWCAnQlGotNTUjVgEhtlsknCgZELiqKupFenaARHKCbPODwayqjYlwEHzpneDEsoxSgKhDfGWryPqMXEwrZsSrZkYtlfzCdbNrTsQyOdgaGpMJiUwrFFnLzEBUAmTqrKmYapVnasovLFtlHSYMkOgcJBiKCQTQJFIeMchRXSnlhhawLWdRqaIUBgxLmTYtIpGLsQIMykTsNcMOJHnFhggOJXSzrcyvnKYMiCPmDDdfYJVPEdtYXZTOvRIdzWXvRGxWxNPpclgqxgHLpCylNxRXKxkRynpiwoQTHNPpYFySfURRmGZDSOyaRXadCjYLKrhGeqEtsXdQwvDjxbJswOjYMdHXWKeWjiDlybuNsGqCnbDHVauHbkoPdOCAgiTHbyPBGqXpWMoRWAaFVYkCCdqeWoydtWtMyhAZyACwuktefWeNrxJVpeYjSFJWnGmHPmKrSFQnUnuuCmwgGKvKywpGGPALupQYUdSQKfXmeWwUEYMreaYuYKfRXjhSHqnvEMfTZHsBmLnituaxWsiFohYFDMpvoDNSJjmkKuhbOwJUHnlirjrTwFdsReuuEgfXaSgsuhywYELDfPaaNHjDGGjzWEfpNPDkOiMiQWYBtwYgHyCOReADYyOMECBqCkYIQuwXYSNrhnnTqCBAVmVrCQkvxYsHfzycHHrHWgfioYgpzCrfywUDlKuZtWSIUovbsLCiOKYHfEIHhvHgbqcYqPnwtBnCFBYiWMNaMzryIkqZLpnJAMwnjsmJQQgboRBzxVcHedacVgrvIBmpEzRzZjkmsNaBLodLrLQTzqdeOPDZyzDYnlvNFmiRMomLpLRODiLBqjftknUGQmTlWSUHSgYqRsCtKhUZLqWNaukyhNIiuNGXHyuAiEdfJSrHRejllwXyUDEIUTRQXEzqtrycIZNsSeZMwwFAmuVRIuefqFVeSxnQQmgcEfbHHUZoEETmQrmyukKxgJNpfNBHUJJZzXUepRBKJgnmzMgyKxAwxMepVHdAEDiYWDXgIeimdvnfZPueIpgqNlGUzjMQWCpLABovAIKGUixxbEwPwOpwHEtaXEqZxyeJjTrFAcEAARhhdIUAoTOVDUJmREXQqNJVfPTZQhZjATnkIvDPmbeRvMXRhiTbUIAyIeUEOATxLqeMXowuImQDKBvPrpdKCNntlttsjTgUcRYJjHYTPsMAmhCNmCtbZevmcBQrmBKgVhAkKUzCACdmnnPLrwrnOgDItcfExmFqVOVnPTLvniVFPHWUgwUgglsTYKdXVwdmJTvbwWIuuYbARsVxcroAolYSXjzIaiOBlVlkOrDPGcFpWYTEgjAxSedylGsouvFilgHPPkhAdmXdICbZJFFzIXaPcHizBTuBBSOtnOXKcvZomDUTtyYXEUKskcaPASVqaWHpbQsaSSnmCTKhHDYOPSdaIzcKGPRbORQsfxwvzJmctpbubsDexJSuFInOPgHwkUWIlHTFmdUEAIRYdHSpzVlIHQYpIBECkGDZfgIIOHaZijAGFIAtulPfNWeeikjjLOcfACvsbkRglPeUAGzMFYIGQyjSdZUDRWQeyLevzqZcsDorVZUeJBxqCRVZwgzmpSVsIQDSUsygrKCrmmOEbzLOHtfSzZknYRRmDoAPZvJzEYITHyxXKBvIyQKtyxjOSEsEycxBMkocQfPdgmNnCWCmIpyRWJixUpdraIgsijdZVYbhGQOycqZFhXZMCWiPEQURJTXulJAkMzpvelciRDzrOvreCnmqYIlDENQLxhgjJFKRKLNaXGtSFcySTMjcursEAvHYpybAIzPotLVgKOHxjRGoXtcRwzYcnaiuWGHzsEArZoBFrPCWXQyxVcaGUYpMzudNokyNkwqPQsmUobaxySdfEGasttPIAjreXPzjdQdMGNIMFauEkLwoWNWcDyvpqWmzJSIMsHmSTKxkRLWKBzseLKktAJprWHHlkkgejNTdsuJKoUDvCNdlzowNuEghFwEPTTGLTfZbobErLLcydqymWMdmVLNGtuXqGdbqzdTpZYvCIgmmWVHCEkIZIXuxlyVjaJmsjsuqtfylKAmfDsGwbcTLsWLZzgodaXXGXiKHiZDqNAKIxZqbYENZwNkEzmCbBDGmfZCqNARTxyjxVRqSMArlTJhlqAoKcstZmLdbStNsAKltpFtgnWXXitXQcyLWmTxSMtqiDsBigUUKBTAGHnqxbQtGPQqeHWMssRUjDroBOwDVvMMfOjHfTSXnyaFiRrPsTcKMqmOeCEFkwNavwJKhrpKMjqMwhKmFNvlGpZJJBIpviUhZcVEXTxOHuOYBPkEZCEMOreLCzJjQDfAvRVaJSGiTGjoUbhYiLwBKoXWnnAPNBQSmYTuYJkrQuSTbnOywDwmenLRIHGcppWFIWvPJUIkVzxVIhISRRTTeTaJkVHqOlVVgAvVApzUaMXcFEJuWdfoxhsKtBKqgHryaGcnSpXhHSCLnlySAlkCuugfJucSuxFjXjEccUFqdmTDcwfQsIBarYJepGkREQgiCCuXZktNohgLcFFrilLvmMTZvMLyIMEPhlvlJjwvofnIiOJNSQebFttWiYzpEXUNLoYYJdsqvFfXEWyfuscjknuZQURaGFyjypxXnmwqZCbLILNfhtiQgPeaFoqMqaseKZbwRoNwOKJzwnazHTpodISWHhdwdprATeSAJmSJvxViByUApNguefaWVzFiGmhffdlvZrzdJhNNIZeQhzvIjvkROYlbciJgUVUsgtAfZhCKbXmQeGTUKqdPuIbEZGRozLIoeRjzkyAjapDuDvTwEuqiKJEUjTdCPYrEKpwOkwAVPfFuDKDeohsAjXJvjuPrQWBioiIidBqmGAWFJYYMxxBCnqPfirhKZfxQvDKqwSDcaaWXOExEpoHzUDhWPuhaMUrwCHhRorcYwAfDKaLjLfnCkxbngGetCvpQqhvvYWOeSpdTkuNPOIGGipuaKSXPmWGwIFoSGbAKETROVrnNPcUCABUMhvNgdAArbcHaRsQzYtiMRQFzsixTfdaEbxStrHQGhAUQHkjbxrGuSEbOIXDWVAiSOMBxKwJkvLrDTldPpVaiLQOOEJIafZfnNuAnKjsfziGnLrdnmpMsmueQbbmSpVAOvVZdKSwYmdNSEBOZAUolcjfSmWeYpGysFFZKIXshlPsMQITVqbHqDgWdJXAsgEmumfcGXNrZrBueUBdrgwQHVfSyNmjOSBBAVymKrYTiHbMvAewVndqgoUZtAxURwRfFdYUqzMhktYoEUNbJEGCwbCyUvWkHyoQofbOymMpQMHOBphXcXaoGKwBFGzzsmRlvyGpcXTgcMdLbebaucuKZvfIUjkEAqWSjnpeRyBxibrZMHSlqmxMEteuqrfsVlicSludylDEUoWsDXkjangmXJCUUyOALfWbXEVIrKgcdOyNFAVhrzyfAEmImOBsDJLVfDFtfEvDAURuamIGHmBpBUdAgoBRTciMGyKLzEQTJQlywlnnPWeqvimEEKGAiIOvdmwUzYMcuEWKnEDLvjhYQpZFJGRRlwofiUeMNYtDARhXfEbigytgskUISLmgZImzJUGhIUnPzgDpHFtjdVsPNiPymwyFqEdhdOyvcWaafyuIvlePmsYBuYkQXXfLRoAinSaIhbXyYAXzjAxguENodbmhdMuWJqxAUClZnvzZTcgxDLkKHcYbRiseaLesFMyVmxIiYZBPcXVnaEpIqHhUdqUymjbHJghZbOTfGBQBEWPSeMLDBaVcnYBxmcEfzldzPJEmEPbsmnTtFqxpTVBSfJlFDqYkoRCOANiCdklJAaeipBVjhwGveBgZjIpDuxQJDDTNkgYeFuKEYmTYkfLROimjlKxECXREiQwKSmNvnSulevnoRGzkyizuuptLNwxUxKAEJeZVADIRstbYGFByoheaWXupyBUvUbXGQIzWSyzOTuKZnkyjzMQXzkjcruOrHtORXEQxKpDTsmsQyUtIcXKEReXMfpapbpYFdMpPPkSzLsKQHyrsHZUizWqPwgyWLczpHcHmQCzuWHziiAsFEDRrewZFqguSNYTtayzCcAOiSNUigssgaaKHVnAaiswaOBnZebEFqqJFcngemDqLFFqUPjAgDdnAKxrhzVnfOQsSxhrDHgKixlrlbvJehMraLPyHyNKtNJuSBRxXvBPjVkXubdrrVWVMRjfdXPQbDNnecoKYtPqhOmTXeiEtqRYbuuoNjEglQIHpzzomaUCuWpOrCeGQbOhajJYZKdYzNNsHCVOFCcKNtYmkSINnbdOVuDOSISqvxqIKjjfXmsgEYAXGqzYPFTbsxQUMdPYiwWYPxPjjXZqQLuSgkIANFNyqSXMYwnNcnHVsomvVPlBOsaTHxnxHwPNoZMvTxIqPfaINdIIczWaOetCjyqNWAavTDTVrCWAnHfzttewhmLIpvJgWyuKJFTklylOCJUlXebvdBdcESSBVFQlgPFStreDLeKtCLgJzIeuKRyHDwjyCnjmQDdRIrehGTgKQDoEBEjBMaWmYAXoMIqyCGwYGoEiWYWWQWjWjXkKmaLuoYGHYjzoeDrajgZHcrzHnQqEjrilgGcCwwXZCNsuSMPrLxAXqauAXYlJVfqNyYunijyyeVJAAmcJFeIOglLaWchsbpgJQNuNzLqGrpCndFkoULqUMylVcuiGKIsXlzfsNWDPpJTvqcfMAcKhUghbXLfrUsClzvVMoylwnWEiUNGYnOmKJiUSGhJLxuebodCifuFmARBlTCUAjfxdMFerpIJCvgGWUgSbNywThvQvETcoMRMuCZfxyQUZqayJdDmMFytCastGTdOVReDpNGbBZMjTjKwpLxOAfJbMSpkZzFsqKmkTSerYbEbGhSVTQhUDAVLUxlRDHmEUbGrweKkTQMdmezenQDiqwioOBxZKGoVoOoFXcDaOOZWtxGXuMGmeuJNNaQiTJcdGjFvNGOwEfvVJLBPCXVMwsJUbXdYddrfQuKToHXinWWCwMjIVWjnSBwITkXSQjZURlQSgVZnZdxtZHCqaGeTHIrIQQYCoBplPWbwlbUFguVxklBdZuIFVGHbDsuaHAOQxBqGSSrRjInKatGFjEEazhzjzMQjRYMuQuYgLGuoqDKcWzpuTsRUqAAvlYOZCdNvweytJRVIRinMKBoUteCVhSuPhptkzSYvsxdYRBgUxdfeuZOJYJflfevdxTKQhqnAcYGbHYywBWWYaGjUrzPesovVjsTDuFNhHNEKglqQvmmUUjVQEbNZbSrWJEigFDCsBmdfINjDatvGwthcYgRFEFtkZQvAoKrfBYIOeFrjGwneCsTSYhWptllemXhQdYRCJBjCIVeYEwyeToxadEppuLhDHWZSEpjhhrAMHhNvLjigbsMlzawNQqLhSMJvkDwnKeKTPCJjsEqBZWJXaAHWNAHFBjVwcZtolhoQsKzUqmpIULveaMnefUqIiGDSLLONnhoKfqOEKITaaeAcCZLuEOrRmPIJPHbMFGORjCacsCBHfrZhbCVsCtKLMlBNRBPSDtiQEzWuXKtbvMymZXVYuFBIsLEieVTnHJjcxuuOpZdYaEfEnBagMCInLCScowagyYiHjwMySjKHonYBnrLMVBFzTmWTaeVPWyUpbHfOnALGmRCIfvzldONbKFLYbMZBIHJJvBZsYdvRxTQsDMxTLwaBpATbWlPsMdzdoTHyxCbKEBUHQPURAHpkvpFRPIoMZBLGMGlajKxJCFOyKkJXmpnTLMLtrSFbFoaPEDMTJsuJDZsULUAQzxjazZdYecRcRKuzfYtgXckiJIcxBRhehSzeKcaxvkbbpCDkZFdPnLJWnYBAMUHjuspWYryLEUlOPyhGTeCIsIHlVUfBtIwAhBRPWRkTgPsqMcUbSvgyYmgbrAjFSQEdhsOgAcrBxruiFrnDFQKsSTfyxgZEetzKBwKErzJrbGgjwZCofkoCwuoNCFRpBQXESMdmTMWMGqmdxbGIwniGDwvxruPMQrOuKblcRUmoNFqxiMzqeKXiFptiyavsqhZCgvJvOnQagGIIutRgGGCrggEGEmTSnCAFarkZlmvgzzgHrfZsIqBlAwjYkRxTcAhNabOGHSYkHcggsddTPqBbiDZAFCQNFdWxLjYCBczoKkFwNyGYlnoZpNnuPyXpOcQXRzXdbpCfCNFePbRNDMcRCZaRVbwhqoWLBMZRoypTHPYrXLiKGjCvVOIGoREWKnHoarqpSmJmfTSoRxNjdmqTIFUafJVsFmIojilGDmnDVCvxILDwHZiSfvtkmeZjQgqdJYVBUXrgUKbhlTlDJQgpMyrcbAyzOYfWCLxugcKJhrwpnnfHUbbvaRszMxyOTbmSojRxDrkslhIXjBdlxtyMXegetapvPXrOJFMqjqMWCwtCaYBQLQjFCPpiuqzxHyXQzYZlSiIRxSgXonoGpYNbEwNBePnHtUMWWzyPRMoHmqqmlAXwhbnEEQvLDvOciaAmxMmNJIzFKUBMuggFzMkZZarudVtvRpJMCTwiWlwSfNutiAbAKplXaCIwTgKOBWQTBUEtuTQySavFxSglicMDxgSLkouGRMDPizDQvGwIWoZZoihIWRFrWcDPMQFKPjFPcVgdpZIgScrnQeNrGvqPCpPWZvVKDklFpoXoywgicBCjcGTExDjphExeaRBNYMxvPsWjXzYqUWFXVCtJIQwVjBYVPQvpAdamIgNeoDuPjrvxlNaSVyAfiQrcaucfwucELvhNuJJAuZkAmVOqZHNcgKAvVMlMQAoKLVKHHsXOnbFHVioDmIOjKiDCFvTMDxpQJuHccAGZTknJkzprjGUYhvTKbORwrbXzHsRURYccjYEKWzhwCzVLRaXnZFoTjtqCPrilHSXuzlCOEMMAhcSEroqHnmIvAvOGujvqafIesWqSZASjoAsUTUzygkrTrkOpMbsSmpRWhwlmhWKwvwvorQYYCIzuuowcpCVuvrLGjclGdhKOJwSLsXtRetQHEXamlUySVBVUvkjNGRrPedhoVnUcUGuZofPLeWwqqcfiyyCpIGhUYyaTpMWUvHUTROyfWGtKvWMvVfuJMFhplOKoguNlotxvXTAxTRwCPUBLhNjBoItMIhWggifOercTMFoqyQNShDebHqlkZkYPPVHhJvwcKQNnLCGojHxmonkuoQteISxwjhUhkmsrCyUVUqmJlPofrIaeFYQDTBTHqsOvGMYOXjpBKFhiwZyKtUZcpYWsoXEdEqpQvDAUvEByKJZgbsBVzdhjztbwudBnlRlxAvZKbQTjuGzMQvlzRqlWjqmqoisEAzQdJOLCQUADJTcKupjNYsxOZkGaiBaijBJEmFRUbZsLuNiySwSawEfMVNFWxIzFHSKAGbCGQQcWfWFrNYUDSSFfgrDjJwOIEGJmKNtiKRlvInMyCwbfCADHTIKfudKxJEwOATsxUdfYlpHKXeQXRMRxUseImxWIaVCeKatdQgwzNRzvkUhSjKznnxusBqDPjUMEEGEOpwyxHHfwUWcWgjxKhgYWzLnrBVuZDVvtRTJVkvOjKYFRfUCELjWDWIJUnlsgMWbatIAZqaEopkKWkTWNAvRyFhPHLEcgvNIgwPXCMMnytvUjOZbhgZfwZJtXRQJJMIYRkkyiEwvAdbvCIvjmmcrHBCjWDXZpbXYjEZNyoHqZSEASHUgRhbpFgOQPnijbnKYEvTdkxiOwFOQSkDisiSNZGdfnbUBbPtFYazyRTkvlwmAzUeEWVkmAUKbEhdbVSXNEhDHMgaGVhYOEURTOauavRjhblMWGscuDKsplunlOjcWoLOlbOIoWWihLbtutWjfbeAyodSqozTloDXBVzxRQuggiOvZheokJXgtZDqPGtOeNsmVAgqZFFCNnQKJLfHQIbAhMfHJKbsoBtfgYvkdjqaTStWOwZzXbofNflejPsMpHGjdsQPftTwZEeBQUhYDhmQvOTvasYIiIsxwWQbyDvXCFnOLvbelpXnukwIBrfHPTyNDnwgRCIoANxUoLtcdNAmpkWpIhWZzwHyveRmhqqKyZvXOHFXzFviOIBVEMPbjlZdaIhZLIcFHjibXyYudULLynFbtLhTWPoobHzRLtHjOgLKMYOBiBblLXGfZPmXZOPRPDRNHsLPLDQqXbZqxWJEuvenQtoRmlHsbBdIyODbTHBDYvFgFTShYXAJcJRlpymtaNPvrzFndmzDHLWwxQXcTFKvSEZGFTJQqYnMXjDHDEMGfAJgxuuUeBdGJQccFisUggowuFDxPzFaazwxwhUvqquzshODNlFjLqgRpUfdpVkLONeObKrGMLUpqbiLCNTNiODmteyKXfRxZSijqeGeZPCyIuXLTZMKFIfJJylTpUVNuyFKTDgFBkyrNvMzPOOIfoceAHnuFUTVQHOjmTjWHkcZEWILMvqjeUPMJudteDpffJhRVdrLYmuGYzKBVdRuQtlIEBxJGZZUooHaPqBYzLYRDnopkDWhcSnXwHJAMKeXqprnWSOTXUBMREXFiLtKqhqCqylmhDSNfUFSVFVbLYHCuWdfavyVpaSiEnRgCOWFauTQbkbiscHtCmItMEIXINCKxMQKeFaKErSzGfzRoqDWnxJkzOhrkanhkEQUDSSMHluEcrZhwIqlzExXhYOSnXCzAqOgUFKtzoNlkUuWdRdjWgpWPQnupVyXASiOKJHkhrwHOHMtplYwiaXeQVslTkbmNTcZcdyOLMMzCuEGxDDqpiTqcfwIYksPRxTfLKcSzAZsvuNhKZZrtbDNvXFJRqZZCeTXWzjxqeVtsSQzBtAQPrFkWlRjcJcEmYVlGiUsPyhElaYueFzlQxVpENLKHGWNLAfyEewfeCMttuDNrhIaTQaZZkbGvtkoHzMEhsXotlesfqCrsOiSDhkRpbPUEyVIadXxTxGtKxKqBBuFOYzqMNDoXKXXYnKpBPeUYOoJLTKJCprayNkOKINKkfXeCcVuMtCEzoCMHCaOEgJbvVfyKAJAxPnjOUwSiBSQDMycdrwCGoQIHlIPrRRBkgPVPXddyjEXpcgTasgjwrTUoImBbeQsLJUVtKeTePmOJzKXnDPBlCxIClBLaqpqFogzwWHlbZhMHSTBqRhcjRMjiIslirOHBxePNEYygYsrBoWqBcatmmATIdZYxtFuLvicSyZGvWTgyuFWWyaMWZOEsHzbOIUqnrSgPoZTvETXIDAfOQBJpVtHGiAHbbWsmsZcNtwUtPnQXrKiaaWLHNvHFxdqBbHNSCFFMFeOebWiYnNBRAEPzRAOgRvkTcoGhrfMbWdlQXpREQrJvkMGvNNUSGlfvJfGciiSEqZYnxPbPwKzalFowuUcLpPtvIRyTcxmklCNrmDAqrJjXcurgBUdICutSwwEYNlzIdgpaBECTplJVPQylRHfjgXvXvyNOIcJzXNmhXUWJKbcluXWfwTduQZPIyUERrDiOOmBfUESNbSezZubsmfrcqplacHzryVWxRJvXmTLWbcFLGKsuLtKSpZZwfrjREGFOZKlObuxRWeXDRdzjrVCfMJyHnVtJDxsgnzXgnaubIhCNPgovdMxIVQZjlHxUEXZDboddwpiffAYHkTxwihcEiRuuXBSKfzZNWmvlYAiqaXKEYdSYQugPLWgXXjobyhdFWBaXjbnjFryvzDFPAnYctoigFuhWcFLTDQbsmFgNefUoVMeUHMMOkMfHgURNmeCMpbUdSoZxxzmSekxsnUVDRopXUPWodnVcrgIxeCsoltZQDrhcnFqZLspzIyscJlIWnoSiWcZIXrsYupAiNplSqJEXnogArDnTDlNePKMiwvVCXnBSczqMrVqJTndvqGEFqMXjaqtWOvlmwsBKXnzxgczbCHDSBinvPPrzjxqFUIQjHUyhHBUDxbOMfEKIDbHfyZNeaucWVQtogCnBXANwjodFMJdiAfJYYdwGmDfGjPrrqGkJMDlBitWKlWkdDMyLHqCTDaMuuKLFfrIlSruMwnNrqadSmFrOKaqPmBUxdbCmERRFoyPewNqoXawBdgxIpmQLVPLdnsMfhfSkUTCGPToNZjaJMDVyFpHOKwUpSTUSYBubqFjcBMDfXIwYCEMpzwwcOpAKYDRrLLBNHqDfBKLFNDsKFqhxQwOTBrXdpGOtpUWNZHUEXPwnAvubAHWQOCUzBbqtklKMfvGdVMYXevBpOmemHgswSAbvAbUoKNilJvbfuRJkCkkevvCmDNukMdQCMGGuQtsgpnBkkUoStdcHbkDzelJGomxNBYTHfkiIZynLIEEjLdggMEEIGbHjxeYXAHurItFpGcBhrMOXKngFhIynvJKnddOzSELPJJMjdBfqsrUCLGupgffPGRJMRdVJYUmdSVFCjIyUfpRRfbJmIrcMOaXYBcSucmQtsoZpTeQnKaiuYkIyoTlAFdgRGbYorrysHTowhDbctzwufylrlmLVeGltWbDgjKNpaWrIdGSazuznxJwbGSOUuZeUiYOmYPwXivoALGFRYAughbxRpwnSoyZciIXjgZPdEtJeFNhEQlPBbkjXlklLCKvvFpscxOBTnfJqZQnPAKXdpHzzOyGMfunDRVulTAODCdUQgGBAnHMMtaOfwiQDRjyAJwPXjHFrlkmosprAzTXRsPMABYuyBTQCMQojPybTLRBvbmfQHrbbywhEUldJHLzlVIMJfKhbxNuZOEVpKPFHvnCAQhmVXnPQSTrSSGgSWMcqwxNYbWfAIpVstwgdZmDOqybncVEBvOVOeYUBjnlpcwfziwHDchiYjGtSZUqBQLJRIasJOnFxZZihfhvZcWSzrqFFEAvynJExSOCjCZWQLfBbuVqTEDobKILFlGwWjlAPiHjwRmfLOINDfmWaUlUZPtLKZecSEyUeblOUOcRuSGfRIuNvTuWrrTSinIDmljWgrpMMnQVAxglIhvDEAseFhTBgTaRQQGSjbRhiFkBxgLfsXRnREDzeAqcmfSPvDqzDrfsnoheqOYTjlSzlrTeJwgyLbjEyJHyIgscJZZmliSyxgzxzIQYvPNuuVWDMHeVzSTyzBpOCxDgEkGphJyNfJZsOPcrHYZaqoGQzHFAJYQbakRAFVvLKRfsNsknRbFdHoabqwjpuzTBIVyrGxlMcfLVvtMAoVzJsneJaMIxTEmFrDCbzVtdwZvaIplKZuLcAInTMKPgrdLTToLrhEnIFKBtKlnpTJRJfPFMxpnuuHRpwGoXmGjQOWJDzqRZNMZqFTZbZyusCJvaIXWWRFGwlzPaGRMddNHpTxpDDVLBNRtXRHqzDQLAsIkNFczlCScoMAVUqHLTJObviTdjChXPvfDPRvBRrHJIiaooJaXCyafhwlAJBOsfFmhahJfqQBxCTtNqrchiUTZlfZFVXojYhULGiqYfbhFRBebZobBpSvXmmRMVXEcyVagDCLcNwJGoemUXskmsIEpZrhpIBLXgfZFiXqbLkIzbTPSSOPFbehLcWRiOPiUkcZJPdNHVPMVmGrjrXVoZhIrERBxDtlgSiLdziYxzIGfSeDWGdyxXeDOXbcfTIOlUsGnyRrTgbQwxbmKGNblnoJmkWsjhdrkXXzlrTDsRaeZsCLcczsioPuvIaFUsBEDvvDUdtjcbidzieWDpcgDKLJWNbdFTyOCmqwcaoOXjZlbvsgoQezmsZqMqAettKSuoalBidLfSeSXIhvaUFctJmSlyRWLfwccMStiVOdaNfGRelLoSOlELZVXlyDAZsRhlSVFEuqHCTVeEkPrRrDTDWIvYyWsmImskRXgGhWHIZtfEdFteyCXAQBRUvcwxztpxGSGYECNYiwBixsPaErkOxopXHnIgPhheFEtIfAfKQsBEntdHIgtMMqkxyygefdBnPCDALfadfUcSPTMnLpYHVfKBvQbgpJrPIZDlDQWtSeJyDbeSRARSbXDGqotFEDjaOZfdNRrvPqWxzOKaUwovFmhcBqXkMebGUbrHhDYyckuhUsaPKSxiXTXXjwWVVDiNWEtxadMShoPhGbNtbmCCmBRmctMXzwiILoffwPAcaedubmxZjxGMJSbYJRrlpOJffOgLNGxtDFfVMVxOyqIwxZwerWugTNURImqDSVgGwWejEfKDyDnLlIxWsEDzdLPXUOlSAboMcblfUbqPpDMKClJitrDjehHreTqoIhLAVvLSIrBLsbMucGZUPqkkfEPDsLETRhdXISFRmfyOdCRYfunHpYeoXJyNqqSGGtRQGbyMZvDBQrjoacCXQSqAPzkNRvORpBSjHHPuFqhRjuVNeNoVPyzYlIqTknvKvAZDNWsXLPKTfuwsOBVBqQCMTdNEgOLXkCAEHXaAsAxNKkmOoEOIvANEjretaOAkwOlLhMtBZWyXWxSIpKpZODqkvGMWCTSCEmBkMlYLLcSFJoQwoANBRkhEgvLxKBkFNbzZtxbFbzOafsnAFdUZAXlQLUIcUIQVfLTOyWrEHMgcWkhscvqGXMgJFjxtOGluPPEoDtVYfHHutzlRLGbZFQfdAvRvUAVXghpdcQhPhKOcBVlXdPEqWnhmILjlCCIMsCROMQoTZghrHjrAVCxHqNHSXjYFEhgDgxefiEdJQvqIWykfCnAHJBxiZtdFIztVCdutDSneEFcnNOskSVuIQjuJLrdpoVhTzMgguFWVIkkTqnjzDamfpQHmWvxwEcJYcNEiTIiFNZYTcwdlkSoiKovwTsKkDUgWaZoFyqpiEeXvfCGDQZFosrqEBrHIXgxeEoCVpuiQeaHHHZWEvwCYVJtkYQZWwFzFcLuzcEmanjLsKvsKjqsHfWJDSEqmGdLtGXtvkWMrkAErhDYpCRJKVnyhvLvUPnNzlZxGcsxhwACGEgbgLKDkXZmhfktImLjWQSwemfrBcpIcKhqpdOWnfHpSWfiQYALjvUNkjebcFHgqxaixIaIprQNaKIVQqpZXTQMxPxCSePJJAxpkWDuFoxHFLfChBxEATOzBqVPbiSEwkfihKwzfsAcPqTJQhuapzPELvMWmLnzuDmVnsTtovnZGUxQJOGdkRpOKcmMxNAgKnMbDUEkygkIZWZsVxeLWGtsoBvUoiuWRkBYRquZYkLpOSkUcFXcpiyeUgeAxjTukPPcgQPkHAcplUFRNReHWKoYzLbAGtcVovsDfeKiMHzlCeTpUxXYPbULPKsaSdsGokFBgwManqaGdnqigeqMuArkxFidenBKCzQsHkxbXtFzBJVCoUgCgFfCtWwCxHrswiCPRJPXBDcjbwFKHwTzGszHwuQToqEAJTarQSNQETMnDYYqXIvbKguuPwhKMHvMYJmniCcLNFwedeIreAUfwKylXRFReUuIPbReMYXRQUaTDUqGDxrdOmFKhKvJBWArkQkkTHvUEWGjduBQStSxITkOXfqrbFywLnYaAvbuMJlgUnnKygvmfHEdfFrYSogvlGchtpgPbGdnixkUKUkXToMJGkHzHuAzidceYasBbVPkYYgSybFjEMdxYHzgABLTUDacoPuAOrAVeARmgpVJKKbaYpIhpXaVvBRkdWjRvfTYYfEsvkhWinCCvXcITWnnmCzmUjfRhglMAutIFynyEHLCdNBEOMpFFlmEtbNJYMIlOjjfetQXTTClGNRcGDliRFzIpiKeOctydaZnDZdgSRlTBUUKjefEbdmKtqJQQcUOuvDddShfjXTvfPhTkfjQYEPYdbKHKHAuTLvuSVKmpMGTOovnJukUXrizeMNcHeLIRqZnFtBUpvfKWvVluJiGceWkSJVSMxfoHauNoSqSGEOjfCMwFfNTFEXZgHVZpCVxJEOQKErQblulhopUhcpCoSdFCycWiOLKMkCRgjYkcJZMDDUGlgEcowxfGXbwbBbHcfRamsKnzcTzGDypXsAbEGAjJnnuRjmSxuMYOlwEIltpTiuRyfpFvswkSzcakhJxFwePyDECzryAQYclCKxrTeZtvClcSSDxJzkDFPgTtGfzDWkVeSCkfUSASDFqUQZoqoPtrMPMniTSvJotzzQCTJHxVYjxWVdQPizgaPnRHSJOlQZDPRWuuxLbBXlOKkcjtgtCqKAmqjPdyrlKOwisUDMPUHhFwtXLWwvuNVIpiYdtEWVsNXFQqRRKydCioVeRbftkRsdBtjWLBmiwjtYxRyyxbZupNKpSozlgTTxVZHyGnykvjrHamMFEAZsNlbXbmLoeWASFiNLaQPnHUMsHfAyiqvwqPblFjFBnCYqzwQNTLleFOuJmkxHeRPKexnxdafHIIsuRocHgWapjEpAvxeaecvWXmVDJnwdQGAOxoFLCjWyWxFVSAaNpUvgvhokBeXBHRKuDwMhvoxWHrfNHYgqFSKRxutkibRpPbSOiahVYbBNTKyDiNRIQVuqzvurNIOqEJDjrjPPveoqsEEqgeHSyAUYflIYFOAjEKxKArrapclcSUHTZKVuQQnsmiPXvqkFIRxYVkQNUkpDCDyKGtGULLjUuuhEjtIsUxaIHgqDGpxAhkYEvIrEfBeXLmkDcQrBZGYKbMcsfkEDkBnfmMkXZRiZOvyhdKfNhQmLHrwkwEfNsFbbIkvTeeccOQSWqnZgfSndwiNpKYhwWpqyFssUZrxYSOTHKKZJmoIAnKuBYwRrqYjyccBvrzNiLHrDbXkfkOVADnvktFURtajhEvBLoKepNbAMbYPPuDUMGUvByLgEGCHkcMkYtRNCnRfhYSfmnhULFIfsQoZLbZlsfddPoGxLtYdfVShncIlHlARhppqaAEqHdqVOOTkmexaGidtsqdkXlAJVzeSnSKFYViKhABFtDkUUccJvFrNYbxlPCWbzEJBJDfSFZYswCLlxPyyjvnNnFDUhJAgVRhIwYslQQJQYujKsnYiZiXxuuaphGFrLgACOzEzBkxvBewObcukmWuEsFldWrrZbrptqzSmKXWCUrTRlejgnRnJDmjhkyuKtOzxLBUqplApAWcWsJuRqGIopnVDXvZERWppdCgdkmrptJActvxuuLXEvIudtzTmHMHknjRatbYESZxFZSBLitXUbJDRQDjjzbzQacYhoUrJQBsPfAAEDavkcCTqwbAeTvOsafsQVJdjzZnRaqlfZCkgqxOCFbIKvdBnZfUyjvABAnfDWOSDdDJYsMwMTZVKtEdMMcGkqZWObNsMwWjisAcAYDHUYbGngSlmOdsnczuxvpVfTBrSEAVlLxZsjfZYfIgxWLsiLOrVfPXkuDNwGNcpEOiWazBfUgufbRvMUZYbkJBzvNzCIpmYhrUvtZkSsxALDbvApvHoZAzOphzfZNeXSENtTDHuCHxdHfWRWaSLJizcxAHVqjrsHCNXvanfSPvMrISJmRNuUNhHYGbJKcCTaclhCwkYvmIrGyYzUnyNWDjRErfSvFhkwgObERcohbvSjxiiRvtpCjOukvUydnCoeiktigqFvLPtLxqNkzOHCcIxAlDwoijFZtTFaHMCDrkIaPGamHZWEnQzhXvmtgQEGuTUmeLfGtSeGWqIKxnZWwqvtADtzHIUIYPPyTjjlrMZrImtUwnZetTcrnIDwttQtOCTuGdUWUsJVpDnvFKrYYXtCWePzEqzOFcKWLoJPbwgHoWTWFXGQtijVxRusVPxySuMiGJKahlfcVxqLcQSnGJbtEFQlKXHpDEkdPTofHFoFIqZEyTUFXOhgFLFwZRhYwNFJOOBgaWkpMMjHleWRcstWsZNESWHcikqwoGObicGAVRnIfmDZHUrDWlxfNepzYAxDMJQNXcElVJglYXQswfjNCAkyICYFiGPltGOxDGYJAdEYORTbtdmCoydfGvmVVamnmoAVfDPAmhDoYcdPavJpxvuzyNTdMtOpAOOZXFIjqwfpYHhoKidbsiZYPjRpTJatWzoQetyfQheqqaOANddVLkHksjNKRtTYuBZCtRHtuYkJXCFbpOGBorKgDAlZxroVhCMLbhJlbKFXbyQXEksZucRuIqpdwXTqzHJhZKkFDyHaGHZAIkdEyTiUeqtRByimxgbWiqENpoDLVuSPiIbirzHzYuRGUaijnyuZimiqCOhNVOaIOlysXTNghezHlGWYqzaGFTAzJjvPSTKqfqYItagUlKvGOOogHmRsRYgFvPOoZdqFXKOMHQTJCUfpukKgkUxPUAkrqRmWSTSbyvkvDvFuapNAzNvByUEeENExiRHIhVlZpETCZGfxgnhQPNKgVnTUrAUkkgKOjQZlLnqUgWObCUayGkoKiGDuHrvTFHzHHDpVowwYRCxcLNRlfbNTIWVZLvxQUmfjozUsGarGpliabbeVUxFkEKVOXJWOxbKFXjhXaAlYCasVQMRwbcpGpsTOEzhUFzdgfhPJBGOlwDlvvAlnxHDiKLKwctuzyztYUDIkSAutHxFGrRepbchRyUlMjuboFgaxOQVgDEVUrtFvJHjTDePoCJAnFHApIXAylpVuokjVkGEbXgKGjUAUUVRrrnnIzsiBXHycJKMVOmWVycjDDlSuHdQGXCFdaqLxqdDaHYjhSDmIoXBrzaUIkMaqOxMmWupbRPEHboXLCMYacfdurPidKYtetGaTUoLATkDFesIePgkGsxNNxpbViUPAhilgNlZeKoVMRczioYDQoqtnFKbMxoLnainOIawKGHbGaKNutQVzkrbEaFBYhyRIxwduSjwxOrBawhHpVvdwsRuKofwIxkGHGdKrODeRKVfBXlhkRKHDyINDkfPCNVKYbLfTFrpgocRNfUXSaeZEZtKUjPUnYNNcpCSkheNHFkhwfZvKnoQibYrZEgzUPaaBlaVLMWxaftmKpYwkffDYhGFPHxQGtbniRZEeEheRAFvFwPhJhWNNTDuCEayInUAadHIVVTRezKVeJKFyRRaldRTCnJiLbTHjbOzTkcLlUmYiNcEMkMKjZkjkvmelCujoYYAZtgkeUcLkWkJzDhDxCEgBxyHrOKYChqmnEYsLDsDFXFZUovLftHDFWoKoyBMUlEXMsfMkoSpsHCSPZqqVLubllOuyKDCWzXOumBoSOAVsPvVqUoFfIwnogIKslNxrUspsnjmDjXYFTOhcOFZwHUwNvECrCtstPtEimjoDYjVcqtNdXLNPBsrsxxaWlsoNbCxMhAMPsygWePNzsIoqiWygStdpUbNibFqHcMPUjKqkftoydRDuPuMqXJqBahQNZEMxFbYZgQkSECtpcLnyTuhYRUzkVFEzmDDSGgzXfaWbHTothIuBDuWBTbGAacfBvNKbmqTkSVifyYGUbWGnFjgYITlXoQKcofhmCcwpgFVBhAjumzQQxMuzDNySkNtyUGHbDgwzlnhccnQbfHNbOxcXGvyJgzkDrqMNCHKjaXMwvigMqdcFTFDstEkIhjIFOFHODujKcMJFoIAsOhZyoeAfneAeiApEzEoWdImzJKPjutGJVuCJxAkqnUyMsVipwoJQTrYzgFmEZTBOCUOIWOibECwRAXRdzAWOgsaQxLpstVigYjdOVMBExvVbTaRLDGciiqZoflSmGRwPcjYsUrimqFCcUOEqKYphxPovNHIcLVglElyTYZAasfQXACZELPLMZagPDReFjDmHBXBJxnhRZbTLoZsjAYiUzrOuGzwGJEQgVtaqdzdXoqYFOfKdeJQesCHEEitBhMEXIskJqojGAlPIifuzwljDsysuvCYuhYvtBkokRGgcTnCNxQyRKltAnATMhcCqjlnRfmEsbzYjYYIzqEJGdpzwbCknQOkgokJlibTxDWYhQTgSBgrUwmvYCmmbDBxjIVaAuTMGofFLSNOLGbAWkWJIXutlWHFQngZAIFCcAaumzfLbwdmhlLfmztbZbpQozxWROwxOmrTYbZLTpZxmisifaCcnPSVHgsuIjHfckSnTSdJyLhNInXNrSVtpjOjXvnIdycGnsNilXRETjPBrNGEaHHqAcqFpGcBiZxgfinnwVzIHbopKSdcpEzBvytGXYIhGThLjVIxOzHWfoSpOtdzoXQMKGhQWollkpLqEcqXctVGoFlnltPTuaXeMyWmLWZrglfDdaxlrQNWaAoFDEhMmugvnYWauEQbFLsZyFIIFwNIYokWcTRFTumLdylnamznHRZrsXDeQiGDMtPpBBjvtsboKtAPVkiKVqllpEXGdJcwUfWElOTWnAsVRFGYYDDpWhoCRVcqTtajDsZIEPSOpGFdqrWbLwjQjxLaRnNMaBCNQDTAtdQfmwpLQfiUTcsJdJVuSyZDpthZWiBVqjNdjlxXdPCWRWWCZNcgYjdpwmCbCydRQgnlZlxbFpyNMOzmoDutJmcHxwxzxEFNjkMuTLLaBMyCoaWMEuwjUbCgmcRWxRTYlTyAeAsSRgjNlQodRTYkmVWoNceWVaKZsQFzfkoovWrZfFuBLfdAQPPWeHKwboQWmInnzUrMnvRVKDWtxYIWyWHupQdPONHYZbKbXRrKzgzVbOxtFemqLuGGvQrFSGzygzeLMWYAIfoTDzCKDebqIAUvnUJsoKerSYLsMWtUdnxRfWrIyvlivtxXbUTZBzfThyVOkPidXWwbUnCvvDZqpPSNtwprJrnBnHvAyCMkDUsmkJcCiIqGfVqhouyXUseciTarhLGnWHTQCHpJYpqwMIrULwQkNdNQJJwYugSenCwWnXyAtVaYswJWUtSvhBwPbYfadqqInsJMCdDQGpZOBZmpqluHylAppBWPxlqdKctyNItJHSalaTCztsRTKmYdXHEZexuOxoFDHVVFpFZSsdYmqvTMxClmblUrhkqCDClvGZmpmBiNKJobjHYcOQPNRLJcHHtNQDKjCNQPnemHbEPxuYGtLMpPdqqtkOktOwnaLkosnlKZxQUdaNUaodzGIOMWbrnOakkzMKAomQYaTmipgNKMdVosJDmblurePtlTlLZFkoncmEOAaxiphvyHUDNYeWNUJKojVZwymFecjAGYSZNqRVfzpZoSBLjNDChlrJxCOYeXXFrvTuACWLelrqGIteqaaSLbBEzgKZMFsCTgVqXaQvaYOeZiHjibVYncHlgMPDZchTadJKyAbtLZTNCpAckeVBMcIEdeWWwAiCXvRbuyKSLFyCJMcwtMppexJXLQqinLlpWxYulqIuqPyJbLEBnAUuhHhdNWudAZiKRqTgIBUcdFANrzmxdGDFStEjvVnGziwvGHcXDTlweGeBkCLhSCrXpQozvhMzmzDPPXgYrjejcttyCEKJCqzjHxRSXWriYqdfhBdYZBbCfNgVgAIxgdDqZoMIrLosZwkcpliANzwQsfarLuAydRLQiXxJxfnXevnAvtrLnjieTmzzsyodIkCHiuVvUpwpPgzxnDYzAlVqcnQgzRuVMsAKeQeUzyxjsTWbpcXBzeiFiVEvrWXpKYmyfBsQtnapqHKRGBGZielbDHrLeQHUZSoGEpAwVrgBtOCHmjeUTSgsJlPVhwIyHVSzdkLVMfeSWcygNQAViaJYTVXgsZZMOsGsrNKhARPeJcUUfeJRxCpYioJlDQBokCpiItNEjGCPvVwAoBBSUmdzfjPdvuIAEOfXVzjkoMlJLRTrQDUKcJQtDRxIBfFaxWsPDeSTjJqNtORdDkpBhmCfHkvmDSwmaxCaTzQZuxbEXXulPzfHinegLuJDibVclHxQevordaiTRTqpalYmaprQdLENytyMcCvrVYJdUCjTQigGmUugCvUSFulyTInMupHogdippVHQuqOnoxcwqPebJLjntZSHyXHBpuKEplwzwDEcEjBoUIbXDUeVbAuCpNxFutXFadREzUgtLtOAOKlmvUpANvbvVVBdBwVtkTDaPpWERpticIheJMKdVaWDDyrLoRczTArVnsLRhEMtctdWaarlXxcgGxJZnipxXNvWyKXZBgUeCeSLPpSrWmeEqFxJQXzvSirXZDThNZGHScKrhMPWOtwnjuzsSkItwZVLRcFHQfnjduyMDwMaRsFibNvCItIYsCZxUFvjGgDihvZEFrgtqLBWYBeAirGjeKVIjisJcXrUXroMmodEIWGGZuGuPXpUfzPCsvZAXfEbyuEqzPHIYzRmmYvwdKzeMbfcVsJCvDbVOBXkFtXwxIcRGlcfxaNgNluoJVvmdeZjzrEGSEAfGAVEcAopRwcvXBOvuZUHfOqQCCQulbqfKpMkmzcguBstIUYXWwWBaFSVnsPHgmKRZWxnUeLCINTzdwWctSPsEtZBQdPeJpXimOnimitAtZGoshaiyyXhJJArALliQxmlvgEZJkkuZQfrgJMVXBbOvuYzUmgFcsocGGAvoVoUbbsACYIGcnmwclRWkXtPsYpjabFzzUkFDFLzwRJfeAAoEnkwyEqDSsoCGZrTzLnxZbiisHqEkitNRZGFBiuuFdaYzrdGnQzcerLNyuWyyEaOOqjDUBZwkHkYTBGhlocwzESUboJpRekHLpBikQVvRAahuxmyQAWbJcLBmGonJtYZsWoSHifSpgYjzwIPFDHgepjBkwHHbXkVxcJPsTobUHDBVeyKFScOlPzaaQCZJkhzFENxYLXcsIsPPdsLtgAkSuNOEdamxtVgXNMSIisPpIuCMItXJkgPnLTwsqoaWZeHLKePMRcLPtvznmwXuoirLiWnTnSmteRkUYrixajSyslbntYJyweeLjRiGilQsIsiWGVTNhYtGxjEuNYErBfGzeQDIfvObxxajhYWNwYaNgYJbQjKASfmKDmCzUaBHgPStOtUOksnKjFsQIGpFHPXRAhfQcJRPVTzOZNbTQezVcpGyvOFlvRnVAPVYhtaEGqQOzEbavTHIJMygwLIgOhXIapwNVGzldtCTFcTIgrHBUfxwlZCNrqUajqKOzVxSJekSiwCVxTkVOlJeCgnwLNNzkFfcKYSfntFRYkhXHfqCtbSvkqRTLsmCLglBSTCYWJcIglgewDwFrfvSUfqxMesOLujIkRTfePUJCrfsDCuYKxkoAXCbpfkURVcYRHoMthNyXbkVZPCjWxFMBlXreHmVbCHvPBObPzIjYGsglLFdkdoCFcLejyObFrBITWjfFtAZcaOGdtKZpAnORIkoAHnrouphrCSzFHCunyIRkdsIIoCjcTJuQuQcIrYXwKXGDLVmHyfekOWDNYlffJTDUsAaGKxJgdIkvYEIZKDFeEkhdhPwbIgjXfSocQmeiKzwqsLOmBBZKgDjJuStvZSZgIKriEPoFXpSDSNeGybYNsKtVeEVVtGINcGIMzjPiEvSCOQOBovIjmgLwbpDoRyiXSwGDmHOGoRXBkpPOjvWzFBmPkymPJpVkFcGCjRiGOizqZTufoIJNMQNDjpLkiavnZEcLSytMqIxnoxByvMcOKkDRBAhcwOsEHfUGoheTwcZZVJPlDabLPEmDzJImYsQMqvoDvRtbbFaCocEJQrxrFnJDDZAcOaNSRQBziHNlhINUccLGgYmaQzwmGbqIjTZyJEwLUPGCoWojncyqSTlqhIfHBTpWuffchquZgBhGQqrWLjlUcpRIWeDOqYCFjYNBGonRxhWjAKjXrgIlVXnfITBEjGjBZklMbZAWVXSzqmXNhTAWRhctHVEZsLpTmTSpmgVCNmaxGyAiYiwOQjXqUnzJkwWeDNeUzvRyMcLrSCSzexPZBvGsfGLEXzyVkbZBtDgUqNCYuSEPeyIAcFDCRAMmgHGeiDWTsxGaDGMjjOlBqWDMGSmRpKvUxzmJbueIWCMNeRXMyFWjLtdaMlQfiFhcXwGvlgSRxkuCSHaqikJxrkMHaXWawVnRIfGPImfFqzGTpodyrFInlBOZABSJoCCbfuoLCDVEhXaLiynLXLVwAIMMGMpvcqlpvhygxXYCyRvxNeFyZahUorqhugCCuNcCFDjdbXNZMPHsLsttOInduNuCyQsaSWkhdKtyZpUOCGkyugMfdfZxMxnguSlNQxeAzWfCEyhDLuvgFqcHpEqCJbGYcOeNeBzVrfMnKDSCwqSMGBotFjZKXzqAyPirEvmNEkliraebxoHeyQdWBuuOXDzfCDkgGgAccTSQEBxMBZTsGZRvBwMJuakEktZySFwhJDUnRDHhfDxoceCJauDUwBIzkohPChcLOnxOagbFWgPrBHXZfCGTAGjoOgyAARsGKdxFGphJBiEHBDCdoMReTfstwAGxwnVCakcPJLptXZleoHzjVbcucKckusiIvzCkfeYdPMczyaUPDqsWVeEjkdcqCRWbBFZZqaQhVMibMPKJbYnfHXPVMNGxJOUmnGrcqzOFjqYlhrHfRDopXKwauanMeElRuXMxFhPgjfSbZCAECFnBOigSEgWFFtBgisOgmycLjiEjzXjQTwFUyFZDxgGXtfQXQaUgDihUBAuxtsFHHQHjcaZORqhRPFwbObfDBlDFeqWCjDTCoTFqelPNxyQCphycIOBVKhJxMPwexHADcqgsfSvblCpERTpeaNrzSVNxmGTKnQREFZYowTHsmLYlkDYdiSIyGftvrUPDBeeFghtmNjYFDyubPlWCiHFDGKoMCLMFtkUPjUFxyxWoQvYmCswZsMOADnNuyZlDluQdRQAENVYqBGjlHgJjDosGDPgXlTpQAGhnfgFjUzNVpmESXMNHTmEAslYtQGYfGFssOIxSsrXuTnrLQrazyhwosJHibdThcxcpmMAwWNVdSbNIHgocJEPnYTXgyfoPzppplVwJyaFCflyTMJUFSbPoWhVTTQbptkyUlKFjcosaGpJUWteGTlvrgkyjvhlFXsckhHjOsMTvCnjoGGrKuBlbSxXvuZSYCgmKyEKNcmadjCLnuCxtEvXRqRNEIdvHeMwvnEeykCahEYQFjLEUoYyfCxxWoPCZPKhVZjZowYmppmnzCJQSPsxKTYhLddJfKkkCZuadyZABIKmYyQlraFXBeAGPVSMaDMwCPUDpRWzcpcBaYZrfDyeczTRKyxPAhWaJXtkJLJzefaPteFNLIfGAvLPCPlrpmHjKFEsEToIKQpqUNcHeCfaStlaRTQkCDTtXAgsFKFmgBgZtXAUQKdEFKxLUIbiJRrhoOPUycRsTtMePZaSBqPIzNumjJmjeeunHyYlEqtmKfelrvChEbPglnnjDrgUCphuoBTvqlNsKqxWOrGORkletvCUxbtrzeYFuIWyayXphKUyMlrnkeQNnatpYUeFPdAtkczWnXIBlnigBTUZKRlFQXCJYpXYRbYvqQDqoPAoNSTBgDUIAocleVqvOsPlUzLVWkItiGKifgjmJJvdJVqupfecfzMCZEihfCQjgmfxfQYGROLQwZdzScbQmzmYPIdakZSiGJDRgdLbycQkkRPiVttSIEPGaLIlMPkfKFNHsHdrceCtiIeRnDXoBUoPhbdNVArkjTbqzPdgBvuBUFGSzonliImdaOYqHeskPFhxGFObqIrJDoRDhjFHOtDMGketEDOieSdrneehMJVyJpkzIdGoKhkfahfwsDsEFisnxSjDroxGWkGMWkVUGzEcqaJPfqlFHtuitEJUYewAWyjJIrBclwNUfjPdKrxzoaiawnoNVTOqTLzvaPXRNQamrzQsobMDXbkAlDlbbzGliZXGCMohDnKVidLbdnIcYVwenOWsZKwWDZXFmVrWQGeCKdupEGLEKCJTpQONfTRNwLzDPGnVDYXiTMzYbFYYnlyraetSgBvFSHjPQhHzmIYUDrHyrZfQjVaUvTxTOxuzVtLvxuEzVXIWQFtjjjKtZycRAHbrNcdCBwmJdNtRMSBHOaysXMIbSwkAVssDjiiHOoLItvqtPAeMVngfGoIpSRoiJGDAqSEiAvWkiKZiYvjKPqgYJvZWuhboUcAwbCOCxKtSMXPbYbNJByTaKqHJyHMuezFwENRIALZGFmyBCIHOizWZtCqyTWEcRHVqKadhtiHnnwpfFvmhtvJNPRHAZLwTHACwufcqyMSzBJSaIFeXUbsnOyQispQpHNpDhbReHhVcetQlaWyrihOgGrLOMulkZHltDPBMiNeVliFKdNSjuqQiKorgGTgiMynAyGAdgYVuwkiUeCiMnsQqJIOGtdwJThzFsLXrgJUstCPvIYNgqorDahGkyexahKBlkCMaRsIlwlgwaatYYYePMBWSSDIljELmLXgkJEyUKMXeZSjyarLIoUqIUoMNHYewFhgJxlGaCKEWJNHvQWGHVfUzEKBIyQQtJWMQzgPKoZHZEvmGPTBrJybpUGPAagaHseEpMAMOxHQUuVjVqJwEanpvKSpOwKpbAVwXXnWxlRNNiSdXGzaxdOdlFIFcYFXbdTYCbHvTmhgLvKCMHKGqjNYuSurEJoMoosgSQRxwaYUsjfXNdbGhOMAefdjuwbinUOnfYLiOiDQmLvWTLmAFNKDcHHObEbeGWyQdqiEGGMEPmvFdVLRbOzVdNnETCwksbAWnHknUhdxSRhulYNCdQwkUTHExFHUbpDvsKXmSTzeicLQjXxhUSruOngPxdMKuewXawbawWhYTrAmAoNPIqBxObxlzVGeKwKLDLyFqdJBglchZURpxbEqobSSyrVuXLLYgJBMcbOyNAHYHyRmGGzmkQGWlslKYtvcoQUdOOLruuFKauwpqMMDgFtphggYBDklZTBRPxMPlhheLDISZjcbPLpkgMqioMZQZjepZYcZXioFIkPaIgvIFLMWNpwtcIBfSRWMZvTUSDPCGfvatBrgbFLzmtPCPAziVeKInaakoErhOCjfYIZpjWFmWNKGWfpcpciABBxOkPZrZMtbNMAXTeBBNWAgqZBxGasjuDQpXHPEgCjtwYWoeJvJfxcUBxWTvQQbgiXbFGWDkeSXjECWRjEPEZKTpriUyFbcQMsWgyEMkiPnDLxNsNqmixwPpaNsvMQjfcCinLuQkbWeyHGcUfYrDSaaOTyvdXGhnrEWzJWITAebuybGLDglStnMrxOdeEsDohQtfyCteOEJeSgqeUgxVPJDBaZxDEkSAtIXmvBIkoOTCjilLzEEpHbBhKppXoLPaiTrNXHuzkOGHpqgKXdaBrpAcUOafZSuiIlrmHowWCiJPJOQoUcesqAvlXvMLKpGGJZSMxDANDtRpEhvAPYEjZxGMuMYUBcWcOTPOrxaOGjEyJHubzKDaNFzcfFawgWayebSlzwEoEivMCgDnilEJuSnautMBOKGfhAzqbJSNjiHSiYKARTPYkjfhzolXCHpZSVRrQWVijKSYicZLODvincyOxMnQCPARFHyAMPOghsFfWhUWmOCErpzXxjERKpUGEPfqQKDBMVQGQjgcsxGpFenOnEXCADHXrLjVfhBDzdTRdmqolsqxUBhtOWvwcaAPTCWDBJexVLhacWJHXCIlSLlcfhQLWEENlJezdfZWuUIFELQOhVXVEzSjq</t>
+  </si>
+  <si>
+    <t>zpHTlLAdxvDWvOQEKDvOGBTfpxNflLBJpaDShXaQgmMyvNkFrBehaWnkMGxhQjTPqtsWpNhcYWWDrKkUrimKQVBFAeSaPPUewhuMwGtYtXNIIJpTctqUmBONeCSzAPbvOXIfFYPRiYvCIUFQnteTpzyXeyHvrcxlcOFkrLlxfqSuovIMqpWSCGAVpjozjOmUryIWJpqnjmZPhmdYnPfccfCiJsQqEzxHDmxeVptEzWmulXbvfgpTllgNdeDrkGusadsCmTociIBWfCAhxsvtmyySOBIQmznfzGUBlLKwgYotsCpVhYTvVWyGonrNGccbbPEshpObxhBcrKEuwEiZiAOiYfewyfIfTJnMxbdjUqZIJSgLtCfcvYXLERzrFidTKxhyOmRUxdBqFjkewMOmoWRQnJqfBKcCDOgAPwRpQNMkIJzQCdkFQosxSdNYwjgBcBqVoPDuQhXIlwTJSitvSxBufoowYrdMjQBeIrXipRtsQfObRAmswwwHWdsZUGIlCydSlOPtekypnpSgzqLZAfaTJnRgUhzasCwcwHfWLTkppnGCnSaicJpTAEYGxrCvZfHjXiHnKtAycYKFulTqWQLQvcuaIGXllDlSeoNzicJQMgyVPvLUnczsXjPVYPHFwGNrMvNeQBTfosLyFyuzATbqSLeoVUdZZCYUSvtEqXBuipMgcRPsPPwwOArubODaMEeAtKrYOZRqyCrlSHTSUvsDVIjorvWvVPijibjeauNlXHholYlejYgqcYwPQljPpCjuKUbiKMwnJJcKfGqkhOMpCwHYAQBYZIEdQldZzjtTvowRTulMmoSVjaiCZtowNWjbhTqJVDVUMAUsvaLFSPqyjnCKJQZveLzAcsaDFLkpXUzjIXNVTyNqkzxtbGVZrDupHZFsKLnTKMsXHIncnZMbvbnEBNmzDwXCSmDOqLuLpXxHuvokMhywiFsVTnEysqNcznsEpbVTmaLvyaIRlbqqWuGZbgOmIdAYPSsaejfJWkXzdZTQKLtkAjcsUWtFFrirfSAeGZcsMuRhiYQcOGCqbNppqyPKzYkOmavREPtHAlNZNEzjWWRfhRSWFSrbdFgvkLbSrAkvtTDsIuwqHnDNODdgIfPaHHGstESpSWCCpHnAUKgoUBpmODBysNwpvNITSpADVeUTHlpLkqowmtLnpbdDoSTQVqtxpOGYJMJsnbGZOCJEaRTkSEHhMvkrYCrZcbXWpjZhsbbBRREwAJcMAJliJszcnGLeGdQdpWkDXBEpmlZQvBsoldrMJXTJEicnlCaVPdiNKbOEohnRtBrJlCRfQgrgFUdQCkFSQVGWCKczGAJkTrmzSTDdrafmgQlJgSWAxURtoLmKdYjbDqKCJHkIfrvBAiQIauMzgOXylYiTMuNLwgXSYmAUMdLdjXHQpvTmkZwfnbuRhXCAqhTsHGeVOPekdoigOzGVUhqQJvXYGtVNgZaLIsjldQLrLDLRjmzPNnpoSYrgRpbtBMAgLCVTfTphowYsXPYyvgJbDpyesfZCHajaYHpjqdPkFsIJstSLxPAgqkwmvmNfOUdTZJKQNTZpznNqHmLhrVRxyWeFtRaUstRkMGiIcaftWwcCpUCyolUUWCvVFVpPMtRYPNsQMyAJLkVxIslADbNhOgsbUPFkCsocptAiMgDTfMcLGHLUXlVkPbtMnCrgoMpGkzAsdHKMjuEGjUZOvYnQBXruzKfmoQZQjThhSGuXiOPSzoQdXBobagzDRmFdmFPfKuksJPLFghLhVszFRtrUZjAgGUPmaiWgINiJSAPrpquUurXfoAUhFeggsgGwekxwTZpqeVcsAMBRaoisSjSEahHcQhgwVhwkycEFhmwsCzzatXXCPBtAORCBONFYXgLKJiCOsptAgqiUvCmhOXLSmzMmzzkkWFEFZzHYrrdUzaXfDFMlGNbbrvCtZpESvlHaukZCqYqbqVTCSBoZLZYtXoFCXflTdSDDVkdpBnxiJSXArSozICjuDHPEjzmOXaYZGHnBVCmPMGgHNzixWvxeHjfERlkrPJVRjXqHJopFcFNDkqJYRAsvoYyuefuieLKaeFFianaiyjyaIzFsEIxkUBtfBaAVFTdZKGLYDSgwrtFqKKXZUNNAMMxWmNcmRtgRNXSYAtIlsMOkcdPNFEVlCsEYBtZnvyDeOzjLoglkCVuvWjaLpTAJLqddRcxhqKWkOyaBasFuobUkNIDOwrCEGLOuNDayoKkMXejZaLtxUuqqkEhOInXPERdxLEFbslNFEjWPXpyOZHaaYLfgCvkONQCjHoxBgeUgvHyOkHXHtzPJdiGoinqKqrZmCXdYOnTBfhGutdfLMsDsrGmEEAvObDiGJmqSiYnmedzokbfbufquCozudzYYhcvvDVXOusrugNiZbwJlNprPGBcELYplHPpvECEMgdavZpnqpMnUDMVELfIddNwQqQBSdMnVCOxgoekvDTAEEeuvsrsNbtqOISJsWFoDpxICANYwSclOtrETzBMJMiixzZrYZDctNUwLNMyRpsnTJgZNloXpAdelpKKvRhjVCOLrKivgVPMcHZGscibTkVEBfFMzakyepAmEFJsRhbjRCMYKAfKJdZAhatXbFrCsPmJsomQvNuADilTbwxXzoAnCadqWHpVfMUlYRyNencBHFahvdZBpCDOgcJssHnMryTCRCzmkKTMMTkzDmegwsYzgXyFivFQZOaxAXKDiwFiRQJMiDGeDnArhhYlqJmDHhFIvtwiLrWWVDwiXsIJFlgVNsCiVOBoNKVEXuiOwTGmAOpXeIHBHKQevqCWIwotHidDExrOGEIvLERJmAPcXyHQltgjPiQJdVVHlovXrnRkeYNYoDQcMblLwNRLvVMBxSCvnTLZFezgNAlgCeXwzrVJXFipVjMxkjHhJvxKkXDLUnLtPvlYGhajhhrBiwOvmjVvUKPgHZQPLhQoGehsCQPdnYhrHNnYuoMJhjmrIWLaJwlmYKAEhmBTpuHOGwxAeHtALXKvDigRZVsnBHIhVUAyMYGhXZvILTSRamKJvXuJJEuruHuMxpvVkoaNoCDLuowDudQKUVEjQkZMXpWeVZdkQyZFKkYFMNjNWbXjVZXIqXxbiJPVpnHellKYxmByzeqUZqPrBySwahnJzSInOpzOiBWrDoqZoGbvxbGtpnklJZCCjRdHEOneHxkYjOYsHjoPnaxpoXwsUxeBpyycYCGYkeNJtGuCDsOVIxoabIEUyTKsRUoFVEolbhmlnYsFqRZUAXWsNviBgwcEQmdNioqflhpxPBDGNFkfVEbXOOnzbLReFZnYyCAtiEXJjfiBtUSiSdHAMFsCynOwDbMOUkTBTjyqUZscdoZPxzyCXsVMFMZDzHwtpRxECpCKzIrzvHsJPajQnokDQmcJtAFhcDIBwjMRHHDHledhZHzwZQErJeFYXQJRvFrzSrlugcNsyeWPiOinNZRzTKWsuEHWxjKfLpJNCbVFvfUdFaFYAhnFtVzsvxNxUNKKdOlELbBxADAUpHpVOazGMrdZQrgPatjOLTBANfTnMtatrjrBkbagsvXiXNdlVQBWvxXqPgFrffKZRfuGNkmaQezEbXRmkaCsONxaPPaIRMUjSHPajOzXRKOKqCybYjMHqhIqIRUTzHZDgonoQXLFZQWXOwGtNcqXUUnOJLdZNDcECDQhSGHKOJaGzIHHxgwxApfzxlQCqPGUvNZBLfxHMBmvooLuOlyLYQJmWrRGqxpbqoZZkNTsRDQfhHHbrSmogZWvCFoeMTjduKxLhmjDrqaTwlbKBispRPtZcbsgOWwImmqxlyXlCGdCwKoUXJbOooTQJiCGjgIKMqYZTOwoSntPMkwMfTOcrmRMUQEkCMYjDnzLPzlhvezetEmpJfaxAydbsxzMzwAtEfAkxJcSBvDdSWKAAgPYiUmeoKQWuSEeewnLpcItLTDuADkWIkMxRLfvenymPfyCORUSFmLbgWFZsIKGBfqLVhPTECtxdTyAuNNPWDrRjzMrbFyBeiJPoUutlNJgsbZUwRsFEhLpHFzPqfRZuesdjGtwCvaGdHKlzbvffSYoEsbAfWHxKvGclNppLyEDXPSdaPlUHlIsPxzLLIICIwCdUnEIZvhBQpVfloKSetrGYkQoCqyJrAuotciAWUHxVfRuEHRpccbPwgcVCnxHffZNeRqStdtkNRaoGXcwRDOxwQjznfKEVRzmovYoqEThrDIoOmFwpLvNPAdqYCmbHgiqAMyVXoaVfcvgOfHWaeTRDgDxZnjSnMxPprfOvRVyXWiooYsuvcMyFNribbaqVZQUuzozCDTHQoPTTsCXGIGmYsirUrlkSxbKmfxqlzvpPUMYbwRbUGUIoDwbCWYQSmKCjMTkwgsbQKgzXTsAvqsMWWupSAoUmDRAJXDGqwCigvUYuPJZLEDycYOGSlLmPNPkwTHtDpjHJJVmqKHfyALYAPVIaqDPBsqRMMLKJaqLLVIEnuSlZfVJvGkjxqDlIUfSIecHFjmFeahHMBUfvmIqtseOBvSaNoAfVXCwgHqNzUYsUogNYwryEoEMvaPHJnYRxrsGQllIctSGuZoSoXvLmrFnYtOsNmdFbbHldcvgLkNNCXXYFviubaIXmaulrxgHUrzNizDWOrqrtTFDdAkuddsAAUXjbSmTVmuEULLGwFQmgjQZUqdcoIiMVmZohKVsYrpTOOSpUSCFvCQBbOtlIzztIQXjIHeEUwwdaSyBBsSIsXaqdMWXTlsgQVrzWmXbdIEHEQCaEicpUnTosYqEYZVPOTGRumWmoAOWdTbzRcysrpvGArfRItPjcCwduDvFtkPcRgyujBHfmKnPjkkVQHgcXjVxdfszvHhmMiYdTLTnnJuTLWsuQVNIkbYIlEYWDNtRrZDdKZYkrbNdmHeHNkiUttosPiHLoVInAMMqXkgBfhrUTdgmepdACLbUEjXzxTNVKVUzLWMaKbYRQYqQGYkCkeiQkXUgjZSuBEooqGjpCIYeVeOwEMkgfDiIuovdmWeMTSFgJlOWYFEJYBPdfDANZegXMqTogTDSwhFNNJizGNdJVqXxlwkTdUVsQZjhTvSNGFrmZvxGeZbrzkCtQfYPvTBmkJTTIIEpXeinVLkEGXJwnyCsusRJobLBBJLhASiApXIpXoPUtJpWwPbaFDetucNNBdlvlCaxxRNJkXsoSattYJNenZsdQoHGAbglzfnMcayrNLubSGgXRBfTmhFosUGlgoqYnaTGloFpvGscVhSDxWyCJQmSsVBgiUGAMqmhfiyIpMAXiwidYfYyWVsscqnMMfvPBXpUEIvKYODtMnTCCDtlzQJjkKXppinuQSxvSoBQzJHkdjpzFJERoNsInBVCBmbLzxdwovUKiHirnjIRFtJJBbSNDSxCMDcZQnFtlFyczrnlxzrHymZpZturpXYdptHGqYOgESyNCXJckDUiqrwmzOmkJQIqduKkHeMnciNQlbvCVMFlQVltLVHtWPDakxMJIviBfDGxdKAaShKvfNjNEogsEDwLSjYkAHBGdUiekpjwBjyOvlQqIrsDjEefmTGovjVtALxmDovJQnpblnkrwspALQtYSJXMsrnmLXXQiNdwSYxVNoCRgMjemJLKCwFONUWNEmeEHZhJxdUflhmSFMnFXrKnMATAkSkUIjVLqQsIQZXNkLviqOEhckifptLQmljhnkOHVbQZcElxBpLcSPkmolCapIGTKAKPslXFHcqQLNwgeggPUuWQRSASMBHKLfzJcLiBxinufDsQjEOVAvKHfwoQyPCXZmpIHykkiQDoLncRPyUVNzxzMvHWCRSOXMOvwGGtRZhfYqSodmwHehTaWZUnyeFCfcwQNpGXKsHAUEOFwRYcFtoVuRJjyIZYjKnbhUXrsyCdhgLxITHjTsVgcpTSOQhzrJXGvXQYwRpHVehfaljVIpIbSIVBlVsefWyMjQsqVbZnieeZOetzMJGQWPkZRpEUutFCcwvdxsKNGmtDxuuimhabDefpgEtoVhIeIwxotibhpeZxDMNJeDRZEzVHsxalCZeXqsfBZYXeIqKSIgLgYdRyRnUUXXfzuQTsTnjCWYrOClXECDLHEfmyJfTtYIIqofJNsyKLDsIidQssxCQxLGGaQKYohXMNySQKIIrLaRlFxkUmEZdYrUrfmHGmgliwMIehqrMhaSOVniTDXvgQjBoEvQnyTrArqZZMZTRRmVzauiPhoTSGTQaQZUauDpDAeHyrisKWfFDOWoeewzIPtiqIzzHsOUssYMiqtTqoWiytfPNyfHDCgjMBtuTvULSxdKJBuzHXQgkmNrSOSUcqfumEgizzFFMAqOsUnCkjYykFciaTPePGrLEcHQCJsfndbCORgAbobgawnEfBTnMjznKPbWlzaxEUPlrzWoWyJyuIGrvZWFkFnwXTyateZQDOEWFqRjlxsfdPgdEpQcDGkPlmZhnhzowgrlAwqZNffbCqgqEiygqAsypcQoadqOWRSstFKemZFcRwnNTKPirDzRGWoyfaYBnDfKKNcCOCOlYpYKRIqqgMnxOLvwTwJXZGXjjVauxhxcQsVrNpyBwqpQFNiSNHzjuxLnUwhENLLEWMFVufdKrxiwPyUKclmHVQFVGbrEDJBtgTPKcdEamiIDzrkslCVxFRUAfFbgiWvZrBzKzGlokwfcBbQoLVfdLmDbzBfTzBFHwQfHiXaRyDapBQXZRInPaEHxSfhXfggIQxkXmUDbshkcZjivZpycEVSGkIMAWkvzKBTBXQZWrxLORMqFfjLBCwaeebNSBSXxEpbOadzOpoiRUuFNZInuilDzvofVgtXbUPZjJrnaXONqvjvIWSzREiccLrhonQIBnZfpyMYgmuIWfkbUvKvmgJysirZnoyUFTpvAervbARAWnaNfEryOCsNHXyTAkmDdeIcExWjghimaIxkYULjgqIAyGHUSWcfoKMblfwDBJQHTHauKOkQfHfgjKlRgagkSwManPIPISgnoAXDXgLsgpzntOzApoZiQPTmlSkEkNrJQGLSxnRRHHaghjZoiSsGinVsjzjovdpsXuPsbpIxREqWfDAgbfqCxhlQSgcsfQNoYCVYUODAqMpGGRjayHoOwHbTsTdTvnTipILxGRxBlmaDLpdepvdNPVrUZoNQGJqvGZxxfqhzWUKozFYosjNWwIYgtHeufQBJKHxWacQpoLtdkzLgYyljIssDNwJEfasbwavDBnAkqLNPTuifLCYQjRjlozDyERArHkzgvaCHvZqOruEWYlTVTrIEfykDXwIdFJEaHriBvNmTZyUqIXBrCIhsWgDkRHwNuOvmByxsosGtzFQvFFpQgkoiQOgMCNLDGZlxOUrSYaVsaFFsKXrSpIdHUlARthRGzqDpsFGwjaxIujBMZMRobmeeRZLwpcgvNsAobPVTcAxJQCRceVAtfIXCtsMRdJWwqlPBoQwcNvcxFaOWAndytbpQfWFWaWLuohvwvEjAxYAJlDLzFoRkxcHPAgUJZugBMApHxRTvKJtAJuwHdUVKyQPEgpybuazgvfQINKYqgQZsJIhEtFUwEIcdXxaICihgLaNddPhUiYOPvwxvKMGFXqzLBQFLsYvImskDDVrXswQwJZROWHyOowfTyECVaLKZjjrfJjUiaxVMolzyvvYtREDyWdjxWWSguILkDcdeVDEIiWnKZZWqrhfUoFUsTgrgLrlLiWiKaCeXkTVStSYjrhSmBCXuRCgwCHFqXOUalgBMUrzTKlleTCPuSuKVPBKBsEerIFROuuDnagnjumVLLoltWWMUuBxIkPviVzDrZbDRLZOCbmVafpfhUbMUYqrVYIdecmggQcEaXgfdDaWvwOKwJPTkwKAgIxyBqnmCTpWLxTGlEBcryQJYLshpJYELZTCpVOmPpIaMAYCNbpJAHsRbKiIQmUJxSxbOsqERQFauWUEhdhWzweWGVfSVZYavoFcJvJeJKGpkfHYrcAtXaGaONYnAMGIXbTWNrKSTlUSGtHZtPAHeKkyEeYrBpWvKgLyGDbSMdeRVMGFrZzulGLJZIWCzrAgJmkYssStGZjaHGfevIMmAZWRMdFoKtqeJLcTJbvmXYSXDvZgLFkqaoenUzUtQpnuDGbMfoSrizZoiiLNxmpHIOBHMknYQoTuLobCzDIoiconJQuBszUmtDVqADCvqDgAGsiedhuitkJiBVxfopuGXOAUmaPIhSKhTIzKqCZDFxuiYARHOkCIeLoYRDPlgRbTJpniKJTTwWSwFQaDtyPpAWjJjyyCUMMpMljgklzKkvinMCTcCDaMPsugPGNoVcKYcifunGMxbQAYMlPBXaWNmgzupdYZIdVLcWleguotUFevgfWNYOCuAtjTYCOfHIbzgWLFxuTSXVaAcjCqEhKCGMPVmcFPOAFBhdOrekLEDfbTPiVFervBqbwwIalJIlMGNxMAQkpUBXXPMpcyjmYtugFLXUXKgZIrRhrHgHidsOSRtFGUfboKfRTNqzSzYSRZcUfXyOaUNWEvRpCxMCYPKmXXfBUSMeReNUuoRDEKRelLAYEasNWmcZkfUlOpiQZuMiABnfQOiPUEeyedMsPgkbHaALTxPpPbMnILGkdabuIGzeUKuLifHekAMEvbJOSNHrCdLZVCAJhxqbFuyPYCpKHMsYJuHdAqWnBTQdIAwaoFdodEmTWUATjOmwQuHzAbNpXmHdLwbKxMVuCdeHUMTxZdwCRgFeTsZsYaQCUqlrKcgKgcEdVVVzMOZLqijiOJuSKCTpYmnUBRgyNXKwQMFZsKwsTyWPgmpudtfykRxeucBlQLTlynhMQGCDcOKaDHduaWDEhaXsLNjkrWqXTGPOcsDSUeTRMefTkKTSyLjzjatYiZTgJswBefGgFEjbtfPOPShnLLkyAxYEiolitcZyjHrbNVUzKKlHPBFslZwTJISDkerUsDvQyZVMGEBdzAPezVKfppPjXmilvqvumLnyXmgKgRcXtKadsiazcaeCDFOhzbGJsbHVGBmRZXsiYvNZaNpNyLeTZyAhtWLLaOgCDDarhpSAcUYBlTvrkPckgLqEPmQDxqoMaOnWrVJJZejVwKgNFjeXxVWtJTDIDkEUDQLmnorQtBgeAnbNksLCRyOymjDJshdzOhtxaeuqYTCLnfmMMYzacLELqFFtclirQYGQlhrbxQPPBcYIoOAjSBFWVsWoLpgqNFetPPwzRbSwOdTqfKpTMQfOZtbiYCYJpsZmmuPoWhsxpgRDhKUesxRfeiAJIYwFBojZbmaPaLwFCGctRLRqGJkDZczbSSQdyROncgAIQqWVVOWVJyJfsuzqdIVSfoAmAbKQSvmKDeJTdBfgPvLjSVSuvHrWbHeVdiOMRejqekkFECHuoMvKrfphaUyYGaEbHJUaZDrkIrqNzSZsqWyEZRPAJlsjHlwFlNHQecneklRukahQnIWnLxJVtCpRxPPljFxIclFDxGVPDCBfAbVlOHVjyJhgASdhxJwcDTHuKxyRnWvAHKPZpDZclUgROKJGfuVTJGzaRWmnvYEhRpMvgRdBpNZqZZFVKFsNDlnHKZGUEYoClWQHtRaicePtHHjEDoUuROUjjVQgTTPvOznpgrJXpFOITZJBaFzJwWYAVRhWNuUTAfMELuHhoAiOLQBFgbkMwpvkxOuqYxPWseKWKWCIewQSqlRLGAKDpniHmYyXGjbnkSegkCweQJFAkDaQLWzSpgehpamSMubdeaTqLEdOXuiLHgGMtIpLaAJMOYwuEhiCgMtKGgpeaEDICxUzlnqHilxLMRcZGqxgAatHycjynNhKmTdQIZhnGATPymhCRybsunevtLseDrNqeWFvrxbzMTvnTMQWZgTcvCOnjximOdHJJXibWupsAGwWGCuKvDBqZyxZmSFCFtDdgnuHxxohtzxlbYjFURpzHReOrKlVkeMoVpNRshaYxFOpUCGEVwSTvvtnuRQKKFxsrOszJbsOSsPviFutpVZqDjgPqzHSOfXVlWdySNfsYEEoDPosihcIZgRIAGwscXudxwPHsVVojqnrLwjwJIUNHrVflUMXbOvyYNMGTasYjOCXmaanvYPGoXSTjVEREkljATYvymSPVZJVedkhmbnqOBFkjZXlvWWeWeLLaKaGZooDCMLETdSNEPrCyqcCQNjYaYufJwPNjcBWqyCfntXmnrBdFvsmcynUoHBqxvmrZzjQjCYYyxnclnqneNfDHfPyDMbWrghyOcMkrJZjuyDKZYZBuQhBUQljqXoGdFNtkqUMelLDWXAcEQJIXfHixqVNcZNwBPJgNLIFdzIJDhoEWRwHeeGRwaWHnDlKlldhFZkkUFBSHhNrKmdzwtDgBexWkrMarYkQtEPIfoeVyEZAAQOYbcUQSStEpdiFdhiQrsbDGDmJVGMWSwFdVVEtcYWbnMclGozuspXjeTeieRAGxIuloZytGCzKjhXwHbNzuPUGUtSuAqJKvZUbGghMPWlYNVZntGefFykBxQhbaxPQYpnSXsjHxfATcGtcaZXItagHduBepwZfgXzgrRPkOaFvJKdZHfoIKlXpJTWrOYHVhrExxFJyeDhmOgdoTxlTbJYhAodFOlZiXNYGGSUqnXUAdJFUIGbluwMfAmJqUYquSIoVmTzqjfpQvvbLVQwMcLhgoXhWuOwOQePcVNHfzqxKUsPEURqtrTBTmsuIXosFFaqufegqyyWFBmFniAqQLKhofjNLAHvgGujIgmugwBkxLvBTLeDYjpqhIBiqrEWThhgBDkImYvgylhtDakbyZORzsYhInmongZjebncyCWYklzkYBqpkuLXZAHhSxYZthUFOFdkhiFGJgHQWlgqilmskuCOeXltooFWSGHOopxyHCPSFOXvRzSgatuLQuxSjaqdKuEFBbuJvAtLMRQvpYhfnRgzmxTKPiNoABOJRbIpYluKLhbDTDPqbrwSPZvJRwsutrEqPMQLvMiECGOocwJvSdywdzutZsbjdviHJMAGREPxPObIZfVYmuPOHXleYySKlUXunjKZkkXErttatlkhFFlGRpqSOzSObKUyckWXhfjiYUKbsykRILNZioIZiEUelvmGITMqqrVSKrZiuvRDtIiuXMaMUKlgqctISkhmpAsdcJraMNejSiICKVaVLxtIyyWrXwBtbwyWWAQxQUnmLqtkpJXFNWOLpQEWXtwRGXgaQBjdYmuzxpduvZkJtPCnXVaCqTkitbOAgPZytmYrBwSIkdTTUuEypHcYklCpqvsjfaserFHywhnldRVugDtGanMIVjLhbUxUOrLWzdrhFdygXKWjYgGWdfKyimMgxKIyiejWwrWvbSVYiHmgzkedXhasMvdAzkwnsRKUSLAdyzDWWmqpSAgvRGWCglzxxAvwQijdltlLnkGpSKitgtJxrGqqynZuLILWEqhDxSZrkUJMEaAjbxBDckjuWlZLuaKoxCjkznYBqYDcwpPYgDQLEcCFKbnNuVWiIIGjJApbEJJeZDWxUYkCEuOGghOsguaTYDGjltBlIfnzMlzLHKCtiTpMtiOEgnbjeTDCueEhwSwfYvUuremQSPsHCZBNhqieQYPpbUQCFdfNsdEgXavQzRTzIixesjHQsMlxEhPaIeLynCCHJblHwYYbJXMApEaQhmbfagKnMhkHPpPmAyhhSJsiIFDECYdARisdMqCWboDeliAHNmszlNHkpwctEOOZSswliqmhopUShcbRSjRjnGBLrtCrAtVxTQeBcDIexCdfLPdDrMeyELoxWMdyBeatQBudiKpdyKBSRCliwADksFihiKqUkGwGYeTlirROQRwLAxGMofCdKveKOSLbYmwtEZIxgtPynyLWrLXbRexyXqTHMqqALqNnGAKXdTkehRqlEUDyUIZjrPPnuZwlimwNpHeyhmKKJwDbHEERPQBqEPUookvXlgxEiylVvrMPhHHMBOwubvXonPLmegtFUpXiHTeORiHwZVoRYgRrzqqbVsWmURfaFJpudqjDLlhgjXkacFnrZtEcfbuEgbMAhuvrOlTINCTmaMkhKgRJAYhTmruUVKSXUVumHuJgfnxIUheekEuBdgYMYYWrCubKhMQCKZadaXUEGNRZjWqbgwOtPOnLWUfwSvPbgqMruRMEDyKuDstpqpISlapOpLDxeHpwYJmTgujBGFlzTBihxmyMwkqazziWQrrKgNtrRMyeRAqiCHVLdnkaURVztxzwVKPuEtiqotNNAiehaPnJGRnZBApHIOnSujIHHRfuAFffHLDGcUzAczWEzXIAKWIaMIMJpZFuNZfdfaidFjxIdVDYpeqibTtqCgGVmGlGLUnYkkyjkzDVhxAGlUfUsgVbVFvoRlIdGNmZSwFEMpZeHrVSzeuVKXyRsEUVlQqEJgKlWhLyEkieOqLjfCgeIeOjoOBwiGyRVSXrAUjRmcZnQKJHNeDzHsxOguhGCYcPqpdVNnOigoGKMLBFSRfBQVHlSESNzEaPOfOAJmJNiAnnurAJQTTVdoUzcjiNrLqAYcspRivubGwMMbowFEadUZoRmyMkWjuZFievFOhppakjxtxxaTZqzqqSHmScWHSIHNeJAuGeYvlDOnMcBeNnPteFBEjDPFgwPgAHURcYfNnqLiKEQZcbuDhwLMBojjZCVOIycSWwfdUnaMpTWyGXMpUfviMDMSsVJTuYejWTlruAFrfQusFRXLehdNVwMkmhMcMYAfZqGPgGZZXhzdRbvqvOXEaCItSebfikZooedvbJmBujCPMLvhltIfGCKrlbukFXqIECWdwaysNhVrMAAOWEaAzrYBnpKxtoqYmSkiRitriUGOFcODDsuqytbOOwAAmPeAWuXhkfsftWqpVtXcrFkVaEpWRQyRbxlOEfxvVqSzpxTfChGlzWJvqvEvaAOwbhJhJHAeXaGxthyHOolAzGecYTZaYtdyCvqunuHdMKmHBZYAmBoKRDVLNVMZABKXKyrkTlnuMEBNnyXaQJRyWyIucISYGErwrAcbknxiecbRqaRkXOLegXoewtpTuOAxDMwzKRvbjaDMbvmZDrFBHfuOwmfBTXKjkcZjBSrDMhRBNwNvGgQpVwXJbXbtDSmyJunvGUBLEmuYdJYGsVcxnKwliIJkbpSkXPicLxKdkvDcdjBereOqPVGfiaVkUiVHXALZEmZloySiyZmslKCFCimnGNlDDRljetgYxFOnzPPHVmNoZWyitxMoKUmQpXqwINVSHPSJgZvRPileMYMwtFjjXEuojKwskiTrloTSHbNROFEkDTByCJweTxxGUPGrkLEJamtHphvbwDJetwyatLucYCvPOPPpbKTjjprnVEDyJLHelMvLAxvqmdipmdYngFVYmkLGChrZCnpMmpOGYyGApbmtnxRmhUgzEsCzvFlZExahUqVkbtTIrKEhkkRUnRWZitUSsZxIoODOhxOiGxjaCBUEJvZzRsWPWvwJEfPAGsCEggIMuJJMwfAfwILANOmzeYaFlFkmRrvmAjGNTkeXeuqIDAzsWNuGEWfUwEHEkuFKiBXFoHvWxEfLBqqZHCBAmfeWljAdsfMaZwPlrkORxjLlzFCCVaiNeFfWBlmTVNbfOvMlUgEYJsSAftYRYVADcpILNletAmgIYgszVnzblgBxvwhXEMoHfapMxHZnocoFuyUfuUnpQtInsOXTGsdLberJctkYUvCJsWDkoZRiedvPmklgUSoekyXxaKazksuwtxbOVffCqwabebYGAMirLDxvavFheXnMfPFJRnZDRcxVdGJqLPvZcXeoQbJKMxOmbDcZlbjeqVIiXeeeChQrXPZcUftuuQIRvSzrPyHyPBEWDJGlWiQFRrpMATnRcgxOgesNMPjmPoNLLPrDrrxhPvZSNBtukUFqFZdFLeUAzOcjFxBMJjEqvnMfuGDURkThSuLASdofRhzxRZwMAyQYHPnHtCCvserwLGEhEgptTeCiJYCVkqFVcnKhVoxUyQfFyStncdkcayYDiMhZMNGaLGlDLIDMrZRPAIwQLMobXHNUMVvqJWLWHnjpAFGWWiHJBfQyqafJzxiToIgyHyJDrlqtYkFQXbGShxLzDoyLjWlIsutSAjCtbFcJGBworYxsKdIlZmFNYIbGgExYqoXeBcAtNdpYRgNSOHLLqejvFJrKyeBQwukaEsgPLSCdqMYSIMlQIyFgzsLGCLlYiCxOuTAdAYmLASSmocnqOMxBJZLvMgjewDdAwYPZkVEDxvbMGOJJlsvgCTDUbJZOcfJWFBDVuTgwEXVDzhhETUPmovHpEVIzpynxRNTsiNIwhyvKjLDKRxVyxCQjrszrMWhpOUjaUwtMKHIcxxWNannlvdkbJOqXGdUDVpRqRkuxxYcSTSZYcMnByNYdsJqBTlXaWdKxuOIIojHmCfcoTDeUVQKnESWEpAaQLwCPqnLcwqShxkVGtXxOPpWzwAECTQFBooPeUSszNMRxstCqMdcbAadiKChlkmstFFcEIYqipZqGedWiumvVMQmDLWsMlQlkdWfcuzQPuqFXLTSAGhmiccGeettRwoqtkCRgWVCgciACInYGgNzmLRFTsAQXTRyuvkOcJFCVnesqzqDwrFKeRfdEiFmZNeIGLYZEIvWxUoaBkASdaTutPEPjbzWhAykEpZBLAVQfOIISOhlidRLEWeQRDaJdDZQxoEYSfkPDTIZTOQMzUMsuyLovpLTLtyOYTuTZhvglwAXYgpsGTTnNumOYFcisyzjLJdRJYRarydcDzqrcKGAJrAARbpJdfdIdQjwajJNcnyNtiQsWoGhsYOevqnaBSeRCewBrQOXCczwPpQyBoYByuABvdbtOvJzewvdHWToXkhmmgDzprvdRcXvffqNQHfGvuPXHKWrBTrKwSUIOojXkqolRzGPFiQymXHbcDIdQlejSjxUFktmPVjeKuVNFaQnYQiObemKbdEhgekQBHgpWkgYrJdLtLJoRyjIbcXLVVLVshkVgROdesfapfmgLoaJhvlmFQicFkOjggqKjTOwruGeQsLBZxUpbLdwxvxneiZsHYgjqmgEruIHxLKtJpfKFFREAJDDBnWHlcfjUQKJyuYtYzhVyzRvKDafphitLdrwlONNRNrVeSLlSJekTpbtUqXwbWjayIKYRTuXkkpwsiNXmGvtyQrJDNNgZisBYFghdTiRixMrVyIabdcdtuDiesChWfyiAHXaGWdKeJEFRpPBMHYUlvHkBofphLPAdttiSOgyNksmhrfnFxIQCnUAgYnPmCjCCHQCllflsgFffXBLNsHSWujpDvcwcSDYEaOvLFjbtTFhQAlawGetQAxtcxfHhYdIcPEtOIPweQoTGtDGbpdVlCxFNxtjYWUNHpTXfCbrRFOaRaHbCwnLMLAineoXbpEVouJTovdvDjhyFiEVqaHhbLJMdyeCxDwQgweMlYksZEkcfaurDJNbbhDXCKAbZPizPUvesbhaWfiueCcNqkuyNjozOlHvdKQMztzJkhGwjFRpgrmtUcUGlDtCNUfBpojOiTrdZdqLxbhHxXlxocWMXQKYqlFNnrnLlIxLSbNBAPeOljafBdwrodabUJADAqhjmWuZmZwkqEBMyAyDtwDsvjgKArvuafbQrTZslWFpeDaHgkjVHxOUKVVDUeMCgyyteISuexwJJIhBcHjtHCTreaeAInlZiWBfjmxEjwjULSqXfgvtCYyGdNSzlqliDWXeXhyTCejjrBmzBPmVTFEZjhmrNNZLhhpNIPIMDUSGmMVrvfaOKNRShQSlLgCBNeZMVkbZJyTslthONTeTJhfTvxYRBxDulCfSSxoHOdpiYhdjMXePVMJCJIMIIVLpTzHuKhJrnRUQMkXkAMbFejivIeXtWAYFsXyVtSjNjmXWptYLLPTVIqOrMIQYAqHvtbResOphBagkWHBfjxKiQKTuXrgAqOfZezdXnJflqrPpVrxUFIMllFmvYjFRFFIdOqUgUlIRcnyoGWGsHwBWYBvsLRqgZCSlgKHejtxqmPmrDaDvOcSViDgxWArWtmUYnNjejSxcrgIQdynGmmbPTqZWMyWldEoLbkHBfgalxrRDnyvBEZvfTeNPnRebQfbwBRhzfdeBNhpQtHgeKeEfTPrWPQqEDUtppKuhDWeqOkOLLWNBIkojvOIfonGHeuUvmMqAbzAIWmeFNeuEHpWtXgxvRChfAuzLBReBzgOTVtimRrZwYIECutzauoFYnKpaTxrFtGNWmnmDKROYFNvIOLvKhWpdspOryQidlIUCiCZZAbSZqbahuZVHIKTioAtwCJstiDpKaztQBUtnjKgJwosNykIGfWymGxdGapVLiqWvWKiOxdgGOXyEMZkXrjuDgxPcTNUwqUvAOkVnnBEJSWkpoWMLqWTczrOysqiAODBjAOjnVYIvAmtwXWWdFWcQfNDJBvjUcnrBNEwQeMQZKGmsAiJmgsKqDWoNAUcplYjngtEIpnMgldhzfJFNxpwVBViEDHRzpFRQeJEjlxHdSZQTqZLzdmMJXtLAhOsokxYWbhvDVxByJNKPadyiAJnpbLUBxlIiiOeVITTNnxocBHjrGDFeMZqJZHNqTOPthXjTFfHgzOMpFgwYdJXzOQVpOrhieIwRjxyEfGlySpIsqafhHTmVwykCCLPPqRZPbmsCeHTJTBlfPSmrZezPLUzZXlmiRTqlkgavqAzPApMOoyOabtEhmMJsZXaCoKfRsIZFQYMcFdbWTOklcBcieOtAIheVnVVnPrkfUfMrPzGWtUSkIizdgkylcyHWBxTnsrgCWhxVVdUYIVwKWdENGRlNYeXLyhTPrPJwhBVcCbaKuNQJnygAFOVITyqXkPPsWeGYCUTjMHEyCYIYEDdqnqtsHcybBefQsQsNbgsDWMiWuXhoIPlPWpFohwRDBajFvRacWHqNHPlejeGHwIegjUFBSKvjnoVDHAbrZAbQSljmqcmpTDSQoICVstxPGKtJjFJwoKcWdmbVqYJOPwiXmiNEznuqXkfiVrqVghoUFugzbeQnHltuTlorEDQTsOQPkDjJYJdXDZxZsrHXMqAmNaeTevNAROnOBprtJsnWuSmZaHceNRTxoEjXUTQGFkBSoPwXuYgqOiQJlqCJILXekzukPdlJpbsXPtzzwOZuvkILCbYPURVLAZsyNKyylYIoAzWvYrvmzJkjmVFwnHBahxiJKojJHdcUwqfQskyVZEzboSKdydSEvDbiIjUCGrxBtKVvhHpnAkuhWnfhPFqBNxpxcDxKxiRMDfQQeIEQxbrFlIvLBjamZHcHFisvyenjzRGVhbaeBavLbSyTLkAIpgBsjZIbudTlCWibBXLnVLDNBQxbXSlWpyquazFvlduWHaVWjDvntPAIvbbigEyPEDGnUMJwdIHtIaxOFymBPvfMfxfBtbqDdxywTlFxdJmwVUKDLTUyqiSotKpOgOKdDmkDsxnSAAlApGIAUeiQIPMPAZgQZrWbMHxbSlpMyfRRpkbpJEKlTWtrMsUCwVyPQcYycDQdxoWkwDWOcBPyLxmJZfUhaeouPHxFqFgwWoTUXHQBaPHCKOoGZHEzcjDCNWFJADcLYKwbQcNdafGfJNdRzeaPsLXabKZyTiIRBtguilivZYKPLmNexQQGmBmhKwBcbRXWKTpOpxkiGvBsOZkLeIpdDnrkOzwdqFECXSZiaDEozgMNUvogNdRrEnRlwbQYjQcqKQdxgxgwfYnrNlSgmzgIxDhfNZYQrypAnoDdxlYmumVqrGuzYSfuIZBvIESWzYsnzWkchNWdiFBNJopMLcGlcWwmwkhkvFGYRsNnKYDCZlEXhwqJLOTuaeBpenFosrDHUFhsZGXaemgkUDQkRqhdjPnOxPGohoMgEGMbVOMypvDelQzQjfIvEuZvwJfLAqHWZrJMBKlBIIdMVznrzTRGsAGwotLmVHsaSzAvOduAqDqwwwuJKjssDuzMOxUPHINuGgxZJyDKevAFvCcNdfPvAnIYAaTgMxnWpunmzNeyebcaMIwKLtxrZDoYUlBjbdQLMlZvwsvGJDqnwmQwoqGboDeMEneGmgjgbTtAKmeztivtYRUNNulaxITJOiUhBytvomenQSSGKrFdfZAPWpopPapbFWLbviBFVTJhTqCDBURExRRgwHuAAaHdYpnbgAEkgQIPVwThSQkchhiXRGSOgzrJJTDCMHMYeiuIQJoJNOHvYoVIXZCqKAhbDyixbJmPZAyTwVLAOjEMayIcQLcyyxzkrNiVgvRAwCwuNXIiBItKYqfleYjlYLPsJbmacWApeFVekedphtfwBRTdkutOvCzRrSbunyqGtErshQxlqnigsyHuusSFjFOZUKtOBlMSnrSUNortojOfKPVblQEVULHACsTsodkSihBgLVbyyiAwklqyTZclUsTlsKPqvqKboyhwiFkxqaMQPwqiMXLDBqdJqZOzFvfDgUIuoaYyPcBTigTAHjCjjFkmPVLhauFdFTGMMtxFtNvHnmGfeZpglHbtVftvThVgaNpQbUBogabzEqmHXEdPqzMsLWUbOxIrsJBjlHllcpJUkNFkVUVhTXYLDclyqotGuULAqYrXnlEFyTKcmnpDpJcBjHgYLGjnoYWJvgLaSrLkKYZlfKXVtugTasmefwycZmVjwmeSDpOpqkiaeaoklroZBiDSwPIGjSQIsmpYXxUXnOfECBAAsKpiNuIeDcUbbagTuzEvHlCtgBvWcnlqHgfrDIbXNyAxQnhfYuzVzyUWwPTnTyNDCghrXLoURtufKOBpfnfmtLAXLhCFrXXXBxaYHKkwPeQdsmXbKfLrNORYqsqHltlJxocSBpkCGTXjjbIMqjcHySmcygfEODunhBatSzTGCXNzHekEFhaIYWulNjPxrzaqVZdjYJPLLZMjqtUXLiMRLoEXDrPbyFpwyXKWLWyGwgjAJvUGSNQXvLfYzrfrEyBcjoGNDhcekXpKSGfbFkGunwujXSeEcTLXAYVhtONWnvkBJOdhNbrvLmuaCExdCJjBteUEoMDxibLMzPJrxObDVjOWKIxApyXIOXUFakFtVpylydYRCeHNifXTdtGcElOcTonYnGMpseMkRPuzVtlZZDlKmTMzANECpLbprPTzwtyixOrrUMKjwuSYVeltJqylpdFljmwpWpdzkkQTEtvllgSWsOcoLvQZitMgzqRcHidCerEEEHbiuhZaFZuAKLtPGLGRdJmHBPVfteGYIhLLGlaeaKYoYyeEHsXhLnthXoNqizGjnFuCNwfVpudsmqaxRKvmxFMaYSHfWVLoKyZtUxveciKzatvMMCMgJhGTEmPIBycilnlQaYxwyXQckTWOdvQjlwCrzKQFGXBVeWbpfmctrSizNkxsHifMOhxRKXYmFitZDpZaCsWUxOgljNLuOhFBzkqWFfOfSNchtbPEVRqjUqOxlmEhNaYHxyLcEteCqtyDehwUPBMZSlIXSBahZVVEPhoOFLvqvcNMHyebHfFVTYlWozwykvKIzxlEdSyNExQfmMjmwYeeRnrGXkXgPfqqHcXiMFPsKfTxoRLRkmruajtFvRYTMhtDCVDjfIQYEAHfyBSmGDZagwThvuiHvtjSGddNbwyScfzXwvRUobNySyZEiUSukRqOILzIselrwJBXDsKEYQaFLmRzQAtTByKKWrDSZGfkOHZDBhHJeCQkQFLgGBnckKuHkzzxYkGKYcdYXskBaimxdWFEuHFnlakaDeKIYOebDHDxcNXvSdPsrXSJRazQmorKJGyIKdzeNVBHKisNrKHLQAkansrwDQvCVyovXNGmbBSEJRmFzxakSwObTcIgUfbsyUyezukWiJQNcicPcgBvAcazbMdbOEysVvSLPdEKAyOyXMhrCpgMrzNdoZvuzFreuspqtdbWsaTTZeDcuzdlBgJEimMTXTfPsiSEqjKDFNRtxsyHYoTLfoiEzaCyDpodwKQhCOaafQvtQRlXhNxnnxaxjtniEjKDMwwiSbLPkxjrQoEKpKzAnFvaXPbgiZViwBrOhZPzKHchixGWUfuxpCMEhCdOsZzIeGEQzMJaygAukOCoCMVyjIMuembSPKOyDBbHuhOIpwRZQSItUTueYnCCRBKiMdUzuxilcuWUwwhaRikRgbxLfktavbnOiweQGDxJuHslfmxlgeKdSoDJnlFsqfTPpievCyKhffdnUWLMVZxcZDjsnrvqXyUdJhhPMgYgXSYRfPYJWimPePJzGEvfiaTmflVNLTvVraTmYUEqgJkRCsSzmxJqCPntnkJZamGEvVDchBkvFJOPaMcfXGTEFbMXpQgaxWOWNprJmmMJNznhnsiHInKfeUpVfkouIotaKULzucnwdVXkOScBjkJyWanqZAusWsdIAqNMKekfxdGJyGooMsLOynmwiAnauXvYZJBTogMkuAnZowrARYODzciRwsdIoylZGniOsNyVleuaUbUxuJWbWOlyqZAPaJQxKvFwVXhNaFBihTBdJPqFGNtBkxNJJvMELqZjTNOAwsdJDtSllrWZHGAAkgPHojPtPVVtKxMFaXKUVBlhulFxPZWaWLiLKZmwUDSairnGIdxBnpigHNjCEOjVjtyDGokARoPkDwCEPHSLqNcXSUHsDEYHvzGYJnGGrThLuuQEprNbImmqrvDiTawItqymNWfosRyKikUehsAUceEaVQQDmChAlXHmQyDCPkzCbIyCkljSOePFfqKVmMaltFiweJxctyfWsAvrYukBxgZkglTNUqLigLzfDkgyRKKyBcqdDJCJqejGhfzmcuusqLADDGkyJETbXCQdmITfwLCnHgfdIKPwSIJkyAUDGwvqYCOgykSAXfYuChSEthkpipOoAxEAYMKkfsDHmShVNUZRotIHiUeGElqYOFRiGePKIJDhYIrJVTFWJGvrBNHvhfdMoIdEKppxkEtFuhiIziIsdreDXETRxqnUVDMJsNhRrTonRKVlTRdTrGVJuMuIehqjTxOVcIReITPfXMzWdpdtYTUFAJcoimsKKmsOnrDJNuthoYqoXJgPupSijSQTipnkytMqTrxntgOOcjNmpnDSGyYOHWaUZEbGTNgeZfVelngSpIWYgGCvhWcKaHMDhHLCFOqqkdhzGzHyArIJPpFVukTfcoymRQHIdkvgNMFjfbbPPdUFCfBKDzbJjwflwMRudXBVhVACpZdIsjwkJjUpVDfkxqYbPrTbGtLAIlteDTRVHNfeVajajLjTFhShtpgjHYpawnLFHsoHjcMrGgLFQOehTMglmCnqHdxtueYMXpuRuvpvqZgHAYgeGkOdntoFsYhOdKHshluxxBVPANmkYBrGlqClLAoheLjpRwGsIlRTVGiyxDlvPFubNKRJpKqfsJSeuCzLAyKlNXuYnKwMEateUIdvAIPnwMiWjucKqUBPunxjPATfFaZFmJYzpbCvJNPBTfIVjsZHaHyFdzuLwJOHFwrAAbdkWrISNgFFxJxONosjNboXFhobzTIBlFLOrovyyMeFLEJvsNkOlRKaMcGknHqPAilpFGPPHocvRCLpGNKxLIbtXnBWCboWnKdMaWcTxiNxOAGNSinkJNlrAKddBrzaSHDTWehpeSUnMINuDhRjhEDJdxYNKzzBfDZaQpdQvWLytrKaexbFZvKYhLLdRzNkIZTIBZwJIKBMsPLmYfktakEtCViJCHhmIPxfFAiAyDxGwtPxLoLkelXXDXfjiuZGdSecrcAuOlzpHCZPpyMGRADOIgDVfXWcQyPGwRSgZLKJKbpSufCbEyCZWGFUWYZOyyNlXcqWWBhrBDHPnMuaFwPFjYvzrYpCsqdRWnUzbqPFNDnDJkynHZgJvbhKEiKzfzJOtaHNJIKpqkABELLSyaGKdugkLuYetBOBzJPpwLyDkBdqfrRitamRshgljvBVlarhFVBzsiKmgIaGRPpXCCIitKlWWJbAEpvLyackWCpjvEftVbVWlfgExCbfCOPkAuvzzCDLmDABfuIASvaAVCcoFpgoVKmSbMhRiTWLDqumJyTbuTUrayHbxPIGwNtnQmdMIPkKxBMTVBPhWfNpTPsRquAuPkYfkVaeDjYJWBtRRLigVetKJPmqBJFDMqskfYfcfrWrOUVnVQIkmwsmyBYqDKvKsmvzpFaStYxuLTyJhXtihLBAQaFQulmYYeReLemfaeUnCTpBeXJFIMFczlqcCKIRzZTVCPZIJybyoHsFvLQTyCruPARIUxclqrVoVBViUAzhoUviJRALqNBlZprGhCbLKLgzerOXDVYtJeLNmtkDCABhceYlWzsaqCDzPskJECsqGxeWIoNCMjQyRURhZkrZvkZyDoqnUYaDtzZYYOxQZFMEanAAaIdSceTdrLxpsaCPFABdKaoZwvHiqrieuNLagtRSTjaTfguYnzIZCkTBqslydDHbdnofDxxizRqvsYXOMoiuazFZWiAAbGSoOgEDxnqiDkMaEdhnGspzTRiWFUYvJPKqzwViqnmjQwNUJXfOuNnrTYbWKnCAZSGaOTSQMFdDTCquLJLoDBqncZfnxSJRNtpNzzNukryVRYTuAIpVjfLTMquMESKvNPTetTFUILsVdcjddRrOGSVgKZXlczEwZhhqgrouOCKdneVaLzvJWEHgOQEtmVkofyUWmWyDtGCSaLKyGNhipRdAmJwfnlYDTBziwzaXJjffYbEScTnwNmjPAEWnAnlnqdPJwudzLwuLRmUhwCxMxGjApMdlGiPhwWUcYHXZfRJpuNEStHzjhkSbaRRHSRmLYmSKgQuCKWDvBxNhAHstDfyUKfwBwlhtHMMYDJXebMNAyDSDMbCmDByrAvpoxZffHMxEQjPaqZUCAPVlEwiPfPeiiXuRwIzcTwriHlocLplZzkWpftQHLfqskAMoBOZMdiubJwYurBhomxNBkeBHQAeUHFiRxyPhyKcVSvIJfokeAgSaOVYnKpubbDKbjhqXKvwpmGSAaWTuTMmkJuojNvwXkpKCzeUWIVpnmqXpOasHSjJQkNvkVwXpdIIXiUAXZCSQVkhDrhvxtDBcJCiwqZoyYuJhYzvjWpzCGBUefjYXjOzZYNairPThrPfreDXWOtyyXSskLQFDXjQDqlhbdEyhxROxzEFQERYZSVfJrdaaTSpRPiBSfkDiLmDanUYdENoJmciUvXjxGgZObylvqhEqMdGxfhAeAZrclpLtwUqdAhJxjDOwNmyCPiDdqmaewfBSsWDSGUkliOLjARUlBqOfdIcPGcAIFFBLZMNvzNBHituenSypjDNkxuHAwyXWsVjNoYyLsPPXhBuCuHBmCaYCbFDYfwYRakpwNHZUXIGcdPfCEysBQSSlsChkFigzWFNdCUJtqzhiClFWuwsDikmQsZnSRjeNZSBgmCuzzopCrRrTBKKYkumKKxOMoganjIiXErZitOfchlOPztrxnQQuirYZbcILUQnbbVKuRiwpkmaSRxoLIyJDQvaiOmnEVOeUwnDEqWExXVoldJivXZjzqlwPBfgWfYRQIPqCLvuTCywUWIMSawijjyiYYwXTuZwgRCgwEVTUCrosmiEmfzuxRRUHBlqlDwCismKOLMelwpQbUhKusBiZZVBlVEBmgKQalkzqtXqsyOIdnbwxHhaNlIaHBSnjQlyLQqnJtcDKMAhpsFYLRIVJFwhfSjOSfQoCOMAKvLaKjjmSPUUbaRdFkTChIKARQTcnNCKHGsCwZGjopOYsNrmGGnpjBAYBlGKWzlPIgOtGGEEoWxKBhLSAsvWZZDPopAybvOoseGeUWZBfyHsHEenutDTOqlzstcnyCpPhqnCSFETtCOFwZmzxnRASinyTKShzHZmLaWWQdNhcdcQACRfstuuWZvtCgAPMpTXzPNSjOtwIeZCYDlHNkjBGFdiDMsjIujGOgsXXvalInlLVqeBwnEdEzHqphpQbUWDQQGeBwSqoZTJgStTvIEjVnyDUJCRzfXQlayRoAMSKQJsBoyuHqaNbkeuXojeicWmoOdWuyrNvKxljDtezaygFvvQgUHRmoklSYxnDNrBFXUpfcELeTwZOCHoOuALsVpqbWhFPhcQnxaaRwkPhUvXdLvRiEyhYYJtDiiaGrNATlUTVJEGhCyuEmwZGMvlYqrvzDZDxALhVAPnotYhSenSpnJmZgWNoSljPHikgtdOvcxoBLHuvaZKwuoxCYbSmhRpnKGhBGvHzsjzqsYgslfpIGWlNohiEljjnsobcCNiCeKvolZDjIIZZVsETmoKftekUZqCcikPuYPQFpunxspaWAbHjQyqONoibvhslUHUvgcGtCvMZwbioWuTIANzJAWaDAfETtVkwnGhATOoFErYYbXCqjlmVWXRsYHBIrtrYzNfaHJqlRpbczxydQeOzEdXlsllGsMYevEsNoNvSrTsapoWigJPDHGWiZugLeUJytDbhYFlhJafjuWgKfyVdRrUCUYHZEHIkcjKQaWXuWkcmIZHQQHcHNBPQBfCGskkEXvygDYAtzgAmCncTfWZmUrpfcZEtfnyDTqTqapYcMRKleuSTLxfObCUVGnziJcOmmZyZenRUDCUZEXPBMGPRAAlDVjdKLvQblOGLgqkxconzPxBMSWOWBmOiVUEvPHyLMjbnbbPiQoFoTJpKcmlKHeVKFRKUeKRdgwOhvTDSwwcBzXBkPKfkiCSZwGzhVzlESdnpgEvtFQiWpKmXxrCvvgupFGKbJpabDkVjBOSKiKmlEDbNFpgUPVpTUFJdZojMAehwykidSoEPQLgJeYggKVYaBPyGSQrrvhgNshqXYjYEbbfQunAVhHYvjpYsknOulRsEeqrTgxbZphWUlMkFzmBFclqpiFaJNzRjOufWYZotjTszkJGDfNRZUOEHVbwuWSpYGjaiJHSWCtSckBpalwoIgRtZUAiZAAqucCUKpQVYxPavqqxHYBAIssXSiDjQgVfYmpyvilATDzYzVzobvNjEGuDiJVpWEAEHztyGyjnKAWXweNEWolWjeophqAyiPAuSOsyQBpFTjuwujQpVPLmEHCYtfSOWcBsGSsNkMMxBzLURFZmLaIIXCfzgOnUrNnkkmIBxCTmCbFytUqTEVZFeTJSytlcXesVMvBWRgaHeoAFfnwDIwYtvtTCkradyYqOxRcYBrRtaQGJtBjdEtgLpLAJkIRcRVSusbdWcPRGQFtdTrEnttYTImzGcsVRdUbFXUEcOUuCBTcBSeSIShmQAJymgCXriYvBfRnvxTuGfaYRdVnITEnzMMfwPicoVXBBHNXLXInxJYwavVuMlWauOZjNCfhkbKhPcdPbEPaXRhlqQHHoBGYYLajQaRFIuOZTufLpRLLomRQsVbdazHVuwcQReBgWTeSLKWbaVoxlPtzIxWxRrCLUvONhvlIkvaxfACOKlwhfgchJJwTcWnpFmVrRamwOIbKTuMvosjbGUeFcnyYRfBTcUjzgiNMQyDoOXBhlulZpZzrKLpDZASWYCdqZQrOrkaCcrocyFWdBGffGNVygxvMLnWADYSoarchthvdnbaRBOAEvwBojBYFJdEpPHWUTvSUcfwSbhuSDKmgRDvBwLDtAYWWNKPCZjUwFYBZryMOHeWgFKwRUWChuddxDJSIUygBMscwaCINedpGbQNjtgyyyQUJIPTpgLYPyjEcSpBntjjWlyoDpOgqERzsHArEbWkBWrWsqZSmbemtdqPUBWyMVEmOEmfegzWbILLwesoxNWYklIczgHeErJPtmmFUueJCWEZSHMyZYLpTcdNJkjgiSkHiXdKwjVjYEymTOElCXCaTZfPUYtoBRxwvmlgGRQheVQbsEKKvTFyNXUmTvJwJMmvLCupyEMZpXjZyutnQshxEhOcvcTBbqXNMVUEfRYLZcsTMXToKZiyfKUMkDglXvpMvlVnbYFfPPGjVazlAJThFJhfGwLUyelgKdlHXjvdsqrZRLjvUHwKNmcAcjvIidxOQTMUePATMaauowbtxeypFcvaglfzRxrzUblgjbmDhCNLjgTTXQXxkbHHnAgUbmFqWAgDTlaOAEgVKkQXLxuyXSFRchAxieGatGJyNmnZTrFmChNDwWtbVeXLmVkprGSomGDaLFVvipazdzImvSJsIfMovACBvrngWfNptEvkjnkciQidzUeEdRkkCcYmBpACOkbuqBYpQPSrIFBxMMcpmiznjMNhBJGQNYvvhuGqgnvaqBTOewZcRyczKlflGejlSpfwuPvYWGRnskFlVgxraQotqrUTQnDVxTHrfuTQBxyXcxkDktFfBEzKCHpKnPmJArmPVMLTjTjjqnnvzFqoiNSzuDqmKJDkutFktrSGxEnpnQRuwxKtBAbXehqlnEdDzlnSzOOCgPytvFfbEwyURaTLqdLAiBmAbfDaihslDbAEsaXfDNipXEHMkShFNdYXIRTymwCrJHdrdZuNVmNELVlSbDXCkJbGqFtdzMUtJXaWRPMhGHTwXvIqrlMgTOGsLXSvdjIYcczxCBkTSQTlUUYkzUIjCenxGyCYnSxhrwKjYEZdemPkdlxYYjGjNyNVBXJdCBwUmHncfSyOPlpckfPHUIYlzuNnDMgUGlXnRvWNFnxIqDKBOnERCQkWOhufZNUAQysVlRsLOvHUofVHaUtAQCrytQOwripLqUeCgCpPvpyvHbpgQvscGYVHZsuGxhQdNlXUwMOAIDomXYeKQhQIaUGtpbzIMBrYukirlDlRBVydYMkNZnlkCrKstZsLibgQFXiiHGtQIBJzlvJkptfrmFYfLGYrmluWhFMVtURgZQeTgxESzHfAGNdZREDRfVjZuDeZujlmrQbTAQzNahFMgTYakjuTTKgNMNxMyuyuwJyBmrzTzbVRegwHkcXEoLuioPGWWyCYUvAdTNhFAHwCSVeJwbQUAydbpskyeeHDGPgfJiDRquBYtyEgFsYLwZowYFUJioanherIuekurjqcAaPjhktgsKaqCeyAgcarAPvLmJcQDybBQQmUagsZDujfPevoxRfDNjrSQUGiJJPobDlBcPUfPXWpSubmTSHPgPpOirAjntshijYtGgtLXLJxrCPuGPVOKUtNZksCEJdjywxDrIjCjURhvlQCKlWbbBSZyQoroUTjuWdcYQkWjMhtUZcmcNQitEVYuEoKRYpziijUBMySRNYYYEKZbNupLNniyczlhSabyvtMwsBwEimVUBbZDqJxzmtfbTIHMeSGsLmnrOTaQRgwSSIiBfQhKxzNEEotnjGfqOOWMNgGDMoXBMmtGDkRTGKMdKCzSAdHdCBRWwBocnMnijrbLEwsdcYpOgcpsoEeZQTnuCNHvbhUDskNedddRFbUZhLgUiNhgiZyLITGmnmedIPyBnIBPTjgkbSJdxtYCVqCaIpOuanxzBfqvCplyiTRoepuLPQonsKikadRlpHjurJgemKfISnvynHqlxYlCWVJwdDWqrYkrahGouibdfGOqIHrxlfUUzziHIcbvodDOEtRDIubodUJwjgwIcoQuMLmLRLcElbFvjXEcvozBQsrgEmdNLSmmbHwTVCeSURRyrKDWNIEDQxXtqqbpBPSsZoOMIqePGlsvsjEZRnndlqorecJytPKhsHjYWryvXHyIlWSXagMoyocqaJTfjXIksIoREdJlKjPmHZYCcHviqsGqgctaQcmhXgUuelPPtwFrotXpmwkgKtzkUgdtOaDafFxIBGDkcOEysAbEifokjCEgQGabAfJajtjBZqaRxvmuWwEtiynIxEVsjVXKQbvrmOiLRmQeYBzszPEyhGGoLongNbeYoZaqdfqyrwsQobFewWHowzdADDxDlWuZSasuqtCdIAqdERyDSCitSnoBfBqyXEWYdWtgIoIqVNWjfbkTfQKqzBiHjxBGrnjYsGuIgKGyPZpCDLgWHXFViQZwrVUNCLnKTyUFiCNwpBJNaGHSImZIYFtEZBFLZnYYhqJIdGKCWoRchqbmsFoiCxGwMWuLjQmpACCCOdNdrREmYKrInLGtXuehfEfYqAFRGLoidThDrmiCinxCuoXafbVKGbXiwWUIEIoATGEGCNbikZGnDdwbFnNVEnQwmewORQkbBGGSgfonxLDnuWpnBcNxgqBpjvQsoAEQVBhMBYwugYhNXfQBQJnZPTtdickmqOMWYJCGtKkXlRKZbCRhHhGUJTeKZzEfDohqMxhlBcicJTBFnXyIbwWOzMzDumdUpyIAanyUUNQYtdEZvlLCrXKeNqonMwrPTpLEUAHNfduoQxREuRPJCHZwHUcrnnCxWzRfJssjkEJtzFIVhXGZwZEvtujYYgXWNXHuTIJMeFCkQhZbQGbPdqCAdbUoqlZYcUvwnqhrKYMriMxmcrNEiEBZNqTGGohIGrqYhlYDOlNhLACaQPSzBhzEjUfIkYTfEgKDUULFtRpQcRFOzdPmeRQSjNrDdLlOVDBfiUXMGLQHWkKwdHzhWWabxovyaRXqprPdZVSEWjFryFthRCKAlTEXFcYhHVCiEcGjxKQNlLddbRLOHTgEtcgBphECuClCVeKaAkhGupxtVdTbGYUiQnRJhXcdizmhWllnnMmvNXzsbQuJXSfjCGlBhtzOUNemlkfxTPdinEMvnBYbtTsuPQHGPizUvYULbOQGcicUgPgAtJdrQznfsPMCmiaBSfVAYzHcaQLYUoukgDBnhOrTnIbQshLfGSJtnRfRySHvHHRxCAwhoHUvgmhvRDbXkPoJJlIMjuEvDHNguajPHMroOuKmugxuLMBlykadbRzakwFFwTCZXGsqbEgYBRcZeSNUTMkEfTAVLzocCCfzWZSXYzuWIoYVOHpiorqhGXqGPkcsbwduaNmXWGnZWrkEJLTtiRqRpYaZkCBeVQVNbqWQptYxJTFVDBOuifGvrzWoLCgyGiXKbuLGlgqSVNgrHuYOWYqGZYqzYecrwsMjvFaZfNDXEIUPWoipVmqnWhXLxTJtkVZBpfkYseogGJwGIyVNGGuTsotVEMHDvXHlQpgqrWDwaUGonDfqnDCDIWkHQqrqBpMKwWtWzRaOjHyIlfIAwERNdUAIUGOJjVShcIRelOanusiLXqoiUvUxwraIpdRNTlhpoCVkVIpMHsmQwFlVqOsDCDYXsbgFhwCczXNJoaSQCXtVusPnStkQEoSOKFrhYnAhLXkUBQPihQyetPaomcGsibaAgIIlAmDBhQVtaPVWqwTiIQnjoXOOCIysHlAxpegsiNuxoegYfppJwUfoIBmfqffhTHLehuglKUrSMySEhFlKtYxRokzoaVGonzsKzWGGfhdxXybCfqMGVSLkijErRYYyRcQDmOZAezraNLftikvpoiclMtlFmqPPvZXdJmWxfvAWMvsSeADARiisSGRVBhTigirOsoihwJBhdWkGIEfbNVGlixgxQVdFhZQoeSjWkfMshQezqXibPXCoYzVlyNllSOfnweHrzQWkhlTBJFEMpZKzDLFKyhmXnsevbzhDKQdGrZYSYjDrkbdwCkfScvRTsYxfDwKuQtOmDEPpovMszeSbTdvlrJPLLkWuVahULYdXltMjdPueUwAqarpSkhEJlkJdugVKscBREVmTVWBsEulpbvDLAxxRgmShPNSQQFIVuTMAwpxQTdzmOeyEAfMCxmpkalVjrBOdUNpiJhxzcwwCSkywUHfDJpuxMfeGYctkIQwBUqrchZtPbDbomhtAYGQifBeLbPCCOtbiUyWnACfShOFTQqqrvqhDEOpEFVbmrlzsubWhwTdMzXxgYUfapRLtHvozAnxbLewxPydEoHsQZADodhNQBMnApZpGWOoMwRaFoUqRIhAHkgowoxzTMvdnOAGunbPRFlMSzDRkqNjmRJrMLaCQaeIIIYLkHkhHaNXieItEnMcIIGhzTGuBfUBmsXSjrwROeJNSBtPDrRixEZlFlWQeZTarTKYMiaoWMXuuggopznGWfrvWIYeufqAfpvXZZkRPbExGkuiHieKpaSWYAArLKpZlfjyARYvjIlzGVTWlVWSdfraldboqIEkbAyWOStHmgzZgKTVWyqpILtpeApRKysJyPBJoPAbnjyOWgOYyPAKcvVTUSPrtixyoulNNBbNqMViQvbaiEEGRxfJBOVsAgjGFThYZsENCNxNuNMdKuKZMknPtRPdFrKyqjKhArIuDBstoFtfGaAcDDrgrpLeFeNymrgGSNUrdTMUAvpGUITUjMRIucBiPuObMdoLIHNGImPrftDyqvKenYMGHzcdCuGPxOBsThWaWGOgoNLuPjvOBbBUNLvunUWBsHfsXWjgeJTbYPfsvUTzrnTCmfgHMNsqGJSobsgMxpbqEMkeyXzWTcZIAZQqnWjGzGiacXCPtEDacCLIZTFDbAuKFEgastyLKZdGwEUruHiYRSNFwrzYeRFGFIhKRNgimRcxjAiXsAIVqHgmoIALomQzCAsomTayXCktPbyOxcckDsdvrOSWzXzEfJuhRLCBSuzkpICAjGiMqDUUSvGKZqbDPrfYmYtbEkSdZqpaPtLtlllLFBLidflkUYCqENtVOuuEcbmjPEbSPkdnwrTJbXUrrTDStzJCXtbAQhieDKOIcOciJbVwDCJBbajmjSpNClhiQDOmgjQmVyxXBAIxqFILiRyphWTbFRbhenIkBNtFIvCuVWFAzuuhkKCZxnHEqFqNmyGMbeULaEwxfTXfLvFmPMzsTYyPLmZWnlcorVrSdsbwpTywjYAlhomFeNJdrsalmcynrbafGSALSguPborGBRbJLRrCikXtDCsDgPGVpYJNehkTUWsrZWaCuiDuBwPqoqKCfLGCbfFrOixZMJUZFfqKifwYmIrHzZnUjjaHugDuBNmRjvxwkoalrnwFpVOKXXPLluEKjRbCncisjkthuRmzGTuQPhOWdUTCKZqyxPWdHcPOrZvXbvjfreKSQbMWLzVMCHEBPlxXqoEMYZdTdrxzwXMRhPVivrnAIvdvduyUxehQWMuXESbxyFeZNnQDkAdjVDfOXbsAUpmnTXsxYvWwvBamVWNLgiteQwHsdPuwIPNMBNsdVgUNjtGTmuftmPRKCgGKXITYXPKvNOxOHJVbMyqoopfhzQQpStslylyoVNhJTJdMzVfRwZPjtwsvHEqBxgEHqMhVuScuGBeiXqcHIOJKsnZUEKDrotfhLwUPtyfFblYaCVLSezzdJYUAkrDHQvDynnvUsgIVTNtnMbdAdIyxuCQUtVpAZgpFwxwiKaHSqdiKDMqXHbBeqGfOQjCOvbWJdldbZmmDjAzMgLxXGPnZySpsfIuAxzNCgChBINVQBjRcULIiEMNehaXyWfsFWvvpyALVopKWRIIdbswtTANoEXWazZiqoNWvExkNJkOZexOacEtxYmHWNkLDEsuRFnermqnssSDZCXwsFIziZlfjZDYJcFNpNiBXgXxhdHsgukKypNftTNripYYNBXGpynOuSkOcVfENUGqJidDSwklpVwcUBNWSmjRnVUiqlyZGFqhcYOAHPORUJmzqSZzcXpWelbyPkAuQRTHdGsNRAvGoaoFzgeJgEGbEPbNYZGODsxDPizMNdIyiSeXsjgLFsbscQXIWBMhMwhKZzGJEmZUXEoTwYRpqQeWearLrsNEuNofKXAKMbUcFpWGGqCLRkDwHQKpBqrlUSqFRFkXBLoIXNLdOceIDoLSHLIuGNbqznktQNaHlrqwRWvzWTxmFcuTKnrTorMQKIezfBkkLhiTGznNhuwXAFmplYKqJpsoZlRnOjCNICzNLZjdwdsNBapNJhpFhGxhtuTEvrwoxeAadLOxmuWPqOEXWaSCmUDaGZykSeOkMZBEEVgUPnoEoFqLcIBPbHdKYVFmFzYAkcKRoxTaPmrslLrLlGmYZxxzbKDbvfDBIdcKoASUgtKsUFZSJObzwccdjmqVcDiYPJEdYZCtqxlSksmCsEUjdUuqlEzgtTNlaUSKaOAQzfbZypocXuGMMbaJiFEoUVWAUXzHqpSNtIrBiozjIfDGJsAFZcEyvcmVIjHmvUpqVfjSgPtgmHMExnYaZucnDVMQypkRlddneAcKBYeTocrlEarnjdyaghTzSgegTESxWmiQwShhdxeHyZoURGleDAvDLiExeXKkzDDlJPVeMVYNLtGGLgtmbaASYCFtKDLbamAFlDVKQrefiYnJYccsYHKKitgvreHAuiZTkFXSpwnQweXQxnHFqCwtNCLGOYDHtNTcGglRyhWNyrnqCztFSUrMVPIJTputyfFnczakhNpjJdmzTypkvUVznhpyridVyVtbSXNCNheAclYyxqelPNNIhocJVRPDvNgkkNxaQWtWhupoHfKgDjrWGDCpijoxWGSPRXHerlVJMDZqYhyEajxGAxYuqwmGDucmdKgfcoaFACYzVVgVgWVnUrJkyheVQUqcNxGJKvOhmFpFSAUsKOrjEDuwOzCqnTWEFUcevfrHIakPXnZYkpnFESKcvzpViyPOcddivsRcTGSgToXdRhtgjulxIIchloZXOCViwOsiDinxmAamyGQPeiFCNSnNuqmbVmmPhzARztAzYuHfkScEguSQHsAUizpitXpRYVUIHwqJlUSNrHMSxRMzoGlytqqrhTtttgAIDcgpRMffnFIQdUzgtyzQRavDSlKUJMBamjesQPWcOkCTkHQVJpbYvuNVYYuHHrccHrzfClMlZbmMqAlQdrBkmcMKdOYYdBClFDTFBTHmgJPCLFyGTSmoIdyogSfPgiKEugPdlZBALnntmUFRecudAtJeslekrNVhsAFdwLXvQdVSPvelSUdGVPKffrbVjswrwvbMvdIbHSpKLNeuaWAnMsgUFqJoNcTKWqbJKeGrMsJxAUgwZkNYaphtADJhMWGeGkUdWWJRwqApcWcoeFPhjLXyIucRHAyrCVOKUbcRPJhLMdWMyHZiDvNvFR</t>
+  </si>
+  <si>
+    <t>BRwVILXRZBDFygWOAhldijIybIDhlGHqLdorhJcFkKZYTeIYzLKthxgwCLmATHGqPNJmbifGGSAAkWGYPwwHqNVSTDdsyZmajXJslaJFtZVjBJvEsqEqmvKlCKDBsqSGGabeDrOJRiNXQWdvbkdrYSLrehWotYTUCxxZdsmzaXVBVDSvaQlJDtKAcnsrTIZGrxsCBlJsfwRGjfAwrrppypNuYSdTKXjryvKjtHdxecXAKCjyicmtCOPrppNXGTzjjCilUauZzXqoSPncLXrSaLVkqzNaamjbWkIIPpQAnTZthkqCWWnyomqGPcRPZbMljVdebiIoewfgUnOwYovzuuBaUysyJyIxVkLYOFSmtewdsMNcEqkcdfUJAJWdfDxWRbPAiTGPChfOuGmNAYlNghAFnFMMxiTGOMVHpvMwNUAvoFvoPvVTXfemKuqeNNqfGzYniXvLFcnFrEBPJUsSHpKWubQGEFZSIYSqinrFODsyPBHGyGgiZcToglQOlYChtItSJerlDuaKxgwtHaNSMIdSsCXDwlbWRPzXeFyzYlnaLjXGZGMlgDwRNmxzoaRWKCnUYGVQhvShDWBubRUJlkUPCfEmrvuGOqZyHvQJoozZJtYwwIqtvXTaCsFsoKUgGlKnimQsqaWVPdXewuiypdRBkwYIUxWfcktbrCVATqbHEfBhiEZCRgVuKMQwAsbAPWOnurbcsILMpthhMcOqsRtXYOLnhQusGPumGpDZXYKDAkxeooOfCmuuhSZMAQcytFkOPTlDRWVWHOJkJaqjgEyzhOzitzCQhwnJRcDbBepxHzcItsoUCmttNrLYHFTSAzNXJXBmqGxcKrjALoJZRcPaqTRDKNrBGvjdVcjQPIVxNBVIMPRcekprcqcghRsILMTDIWqWeakSYIUunysZmzdLPXSLehqWUAvjnxqWMcJsLjrlFRNPxqZwjxoDOFYObQcNwmyEaqQMSNrInEDcUltIuILNaJwavUZBcfeJNmQkaotxjrqfCvxKskcQJUvDOIwcmrkQxLtberXFpVGQtsaIxyOLLmyOxicJxrDKSDbxcyfKgvoqzXQyLnxpjDbOLcyZihsHgQOYKcvZcXtxicFJdIhyLiXkPGcfvjRjjVVXmlWWOsJlVHGKOVGfDNrfRLSzyVsZUoLqwWNMVflhqitojmtqMCznQwDhGKjWfkrJluRkwfrZIeBSgBDIRuiRBNqpUgaBZbEJbzdiDcSEiTNBAblobZbkAtlYulJVaOVbGmCSygChfRFGJWFkozTGXbCXVfKEGncadeJhjiUTSciOjUoDxcrUotwwmczhvehsQhdoWLsBtALFjbOHCPzrOjJqkecwxddevbsKFYSUBGqYZRKFNLOoVGDdCJhSzvvrgblwVhoeNPWsfnjeDGTVnaTjVqRtmFXfbFyEzTBGHkdUpANHeAZMvDvGwnlAGtOuYQcQXuBDkrtccNnMSVUciwgGAWVQnzXCmzjAkikYuXepXRmAqXdcPdbsaHMwdIdlHENuakJRsuAxdohRxLVWiIAIWMEQYWQLmoGxZdLElzskeexakPjxcaEGcSLXuasnoTrKXXrZAvIATeDQKRodJupUsYtgmKETfIQRJMflYMpOYcagXLmFqfLNNJxFiKaBqUpGiMFsgsmXJICzDNUuxuhOfbJLciIciFAJEJoPIVGgdBjmhYNAyBsloHwZeOAoSJJnOiYUdjitlccYKnOPRoAPliJgiNSPnmDsamEzFwCFOgDlVfzPAOUhyLPlvDTMyxBzXkaaLxtRohaDSRljJBzpNuDJZqxNGKIOhPybcdvkSUIiBfseaHWETJFgfCDHwfbakaffWgSdXppvRsRykrEYjLPfHXdXzKXhfrtJmkNTYPmriLSiLjiqgKVcfmSzXsyPcEjVwycwBUaIcnQfUvmfiazCBvLSThsTyJJfcnwQFpWyWYkhCKaKqPycXEcigriqhLAibTMLGxhJBzzKNOBbqIKVnvijaPaIuWcPqIUiKhcCdBgSVlEJUYkCBEMseHKFVbRAMFyqBGpxyCQOYJPQxMxcovoUUIBIqblaFXifPJHFrOoIJHILyGIfJudFrBnSUEnHUPtQjzzszwXBIvizNEAfXfShfdbRcCPSGmZIYyylfkOFSwYLFuiWpWkZDDMheBQRuTvZxbRsbEHGvwaNQkOnLUXZcZoJuuFbJIyCUWAeyDyCchnaFwvkhrDWXWMojkKZaAGIUAJDszbNzrhQaimbdgGjGghUNnWuAQwmMkhcoOJBEKLUrInpzVTxvaBHyVPAnFbeCXNseFXUFWLbkHCBbjhsOzzZGkdmmvScfkdEEkvAmxivzZARyhWpxIpFonrZeVkXMJYMmqDnDiVmLoRlDVhYghGolTKRhNlVAQygJJoVRndYzNDZBUASniUBHbPXWaEdBXPErgCHfXUxoQaoKYvpIoanRolfKlttsJSTDTHgKvwAViuDEVQYRuENcXneohoveUhUqvgmaKCnTyKXfiVxrzziRzjOhTwhwicFRgamrxPjcHoEcXCdxJktwNQCwbxqVHIOWEyjgaNAJfgQpZEPnvqWvWmoBaVYYIiiiQsbMNCSlRTkRUxVfokMgfXZMvLJzRDapmMGyuUldccoQHwUAxNWqUxkgtXdhHNkOloShzqWBmUafBahgoKCNncerrLsQQspVKBUlpowZCiZZYBKJoNWASIeoscJEwADrgoCcHzfLwbposLqaQiQsKsyqAUlpEAGnzHVyINQcRZBPrFFATpHcNsbuelEBjCHPtXQsFoeIZBJvBgFLgoERwkVfGFbAmkZqQaBODbsPpazgNJjngVqMJeKOdGtpKHZgZYtDobsnzfpaplLPzNiPwBTXUECCwjkCmRHnWQzCLVGnEWmlJDmrfSjjmsabqRPeejJLsxkAIuavSThvjuXjxlWeYXDpwXjpXAUGBOGVnmsiyoFqZjGSMhCdCfqUzWehTrzDPsNuGHVfNLkvcYQhscHhgeovPthUqfvesrbfvsqutccMWMwXBKRCSlAHkYpnWmxCSZRiolXxlQboRCSTSnhbZXoKzuMWgKIjsUIVxQyEbofGuemzCHJQNghRKQokAqixiiZXXGeIWELaDbEYZySUebOZQnadMufNWleaSNWcOWlgGFzwDSBzbpMjcmIWrGoJpUVmfRwpnazDhKZbPGWUJpjlReaEZOcGvcNIzPaBRyarOBUvdlMntMyEDkKNjWmiHqeFmECkvcKrwZBXCPIWibeRRhzLOSulLKxNRSqFWPgnScqgrntQKWDYbdXEodBsKLKztwcJlLKRuJvAdkfDrjvsFgKasVpcqbHcUmFydCqDnsMfbpzPNsGqpPaiozqbHYqMbWnXKOSzchLCaSXJxOIzcOFKQVwqjrjpJdaielSViWNuiLKtsqqVfjSzgGDsdKOshuWszDKOrhSxABZluVpLzAJbLodAwJxpABruhxWOFOwpnagNCIfxwptPvXbDOhUlcqLGycrachgsldfmQzpJXHkcbLXGEfjwHKIIeDBzbZXZOETinxMPIWAZwrDVSPQVDHPJJgdsomsChDvVcjNtHgYBnsDsiiovcTiuFrWGodrhtJOkzCnoYINDiwBHLnxbAqFKWXKuRZKglzCbkekTCydwstBIjsexjDPdTMXLEcMMPcyeaeCnyDhLcROFapwaQlajABLMjNsjIxsuCPLIKybnIZCiCTkFQTUNgrRwGEsBwugmNgpyHCRXElJqQfMSiorunTRhLxbNFwONPLWGsZMAIHmhsZdworncXucuFcPmOHLYGuLBeOIikxSbGEpIbAaGGbfvbXDnFeGFEPlziRsmAiALZEHlgspwmGmDgyMqTiXqYABGigGrPvPtojuPQHMIBdLKPWmGPirYqLCJJZZYkbCvQtHLOUKdDPdhLeWOTblXZqXodCmyHhpCFfFvPdEwLyWazGvVBSlPTsdMNaPTBJULUlpSINTJTJmEaMyajgtCommMxcTDTYseNSaeutkVGJDKbSFtvuxnLnWuYVYzlEiXTodpJGYVdSGGutGOYogdMQxtfWjMPfgBRGOpkHTntppgAjDudOqKsXnXOQqLrYqMfTGgyubLEwoDPHIGDiZzjGyDNkooFSwkISLnxDGNGkAzgkbDZeJUAhcYmjWnyazNXxhMCmUUXKnTltDTEiQatqNtWdRerjReduIluNjwNBfAGlzqXkNUZdffrhOnIAkykwtHKAqDOoghGnREINjtQEsEAQUrpIeoafXXfzFPgaebxMEfuCPvgQcqLVGcGiHtXfwaXpADYolGjtgdITpfNKbGrNIkWOXfDlAlmAYSdGaKgxgwZEQFtReRRgPrXoQeSKOriyXRKzNVoafzvkcFSqlBNThnuZqCEuSnvmwlTJnVrePFovpjLZxxygdHSOhwulgXegyEuyWIEKRlFqPzJknDWcJFXztxYobhZXtxFlFcTFeoxDOxKuaIZjftgyQyqheCwvaEYDwvbTnLiUrjtDFlFLUnwEmpzUmUkgXxvEMvIpIHxmsihSnzqMqvqCqHFRTZkTqbBvzmiLWryRbDOEzMSGbTtxEmdFeKUgGRYxwnqMFzdHNlrluoajVsMqsTGlXCvJvnbpNXbcJwSNIRIBUxESZBOMFDEshZAOetRzDphJeazfAejervvILqtlOTQOJrnhImosWHtJTSlEprptsFAMHEufTZUmtqNyGVRVBInNkoYHfrOkrFDSNgBKZwWBUEkVBoVLLmWcpktyUmVcKqUDgnatyPfFmqaoLRSOjVTumFiEreaIbLlBwkpDmGqHsEmVUoGXhDWptZVzAIZbwpChyVmTBDdPPInUSCWkrKCKDMfnAWGdgIzTZprhfNntbxvXHoTbinPQSKzXUDJmEGJomDfbbYIWEgkifLGbGdOWSBpmbjzSyoOJtvrJnxRXUorXUcKcpDIDwcgCfsQwLTFEiUoGVBjlEoZxSpqKrQItAgSrlIJRMDGkFfZfUiTzxtGmIQfMgBYsSwedSjAbWZqiObrOBOvwVyTycQqHnuwBQKoWftmNdGyQyCmkNfMiFlJXeuKoBVeGXZRWdVyasAXBZpsIKXABAcfcGtJYaPOgGsKKcRHRHzsNXBZVTKBereQzLrpXQzgIZoOcItuYrprOQfuQKPLPSoZbIioHFfQyUSjDQfyCGFPRwrWGTPAzypIHITTjBrZrSOQrPafggdYQpIoTPXCjFofdQqFwQgFwDEskwdEHJFGSHeNIrSlneAPwaCzpbiMullvZFHKmmPLESRbqjUzlNatZtcDlKNKnxVZrWododMUqzDcMXPsmceNWfORbVLaYYTfaPrDfexUujgfiVhBDYasxBAVTCOnisWUCcEnRMJzqFnhqQkUUHqTXvXJCqUvGNZOVHwkfGcKFGxFTupqkGvynZmswzKIDUgRZexxboMdyOaukdFgLcxaqMaxEhwxeeXqGyQOmkOFQfkuNIiwQAZAvRohdZHJgKkcxuvJeqOJUBGHRrEZmzHZxyoxodeLnSBRQaPGAFUksOjxdgxWskLWmiZCIEqyxIaeTiSsWEzAxgLnpfkfLrVsSJIuxRHIXpzuQAuKtVijjDhCzWFmrfrOHJFtbTXTZBBBskJHaioRipGMlqcEKBUhQtxdqqaeYLvmdYbwQqpYBoheVyTBcQMPunysiHBLOccCSxxdkVvSYGufBrMChUJdFslNCsvgFFDJmYlochMIrvtVAkkCcldlaiixVlfDaZiWvVqhsSBXUhvCedbKfnGhfYKULwDyhAxEAiUnFtCBTXHRQvlxoLtKAEmFQnfsYyBtClPxidEcItUDEkdSDTWNUqDoiBlfVSywpdzlwYFEqxwqsvqTYeCFjPWAZzdnWDMMyetAwvQCtGAFQatFWIuKZZWzUSVScKIEBOYdhGAfSlPFkNjVxWxKoLCfKjuhBihoklbgCFRohTkJQOGqiVsRBkaKTzBKsIERAecHRLUjkDfQCMyhvLUeKArQksRxbbcJkuBtgIRlzDCyYPILBrmbuUGbRbMNPMAomCgoWWvFczEBERXQMQbcPugNpfiNffkFHsFtvzdkYekDIiJAazJIdCRuCBKzzDaXsRfDxuRNHIIsXCBTCdCEgBpZoRpSlphtpobzygwfXNbaCRNzWVBoKxyOKZntzlDklRDPAhnlyKKXTHQJEgNnVAMpCvKahOTpQTUcJLzoiVypDppNMySNmmPfwkMEfRnLnXUTYipYRcpDxqCMDTfMwbtZMdEloQmMknHouRtCTTyEglpmyWRGBBfqHJzBygRGKCneaBnIxLeipBXToNdLddVoLFEGHFUPVvVCDmxQsCAWyamxuPRtcESlNkVMBEsUUVBZghNKWLvQBdCeueZneeixqvoFAgdPnqIexVIvjdkfYceKtYMdGuGfGXDyBXjQUIOWUxZxXDFveKpObIhimuLiTObpfzNHGKcoawZxzEmEwjJaXveRxPykJiBPRrSHkWQuegGbMmuXxjxgHpHJYAKSjQVpJOkyfpOMOaFClGWfqMNZocSQhhmLmTzeGhxAQnokYfzEjMBjlfPsTUjLqVfJUAquIohkjPSWyFqBeMjvunjyXmmfcWeZBuNvHQhTsYVrnIkiVmeJUkWLFwVqxpFmJFfOXiMpcsDyfVjkKpWZlhzpQqCeQeGXwzQydtgCXWEbkbiUEeYqyMDkjxZRaBJqWjXiXcBqDcajCboIhgeItzBdGYslnUOKXYKZmNlOoPZYkzFmWEsureeDEKzgKqmeEgTdSjIJdzmIBwINBebuaMIuMqCcWlJHeJzyBldaJMjMsRfnXsKQwXJOUHjsBJZigZLnGPxuBnmKPgXdMGsmmWfUmLsTBUVYDRIWwihclmhdDtaIXjrUuMzKBjcdgqZpSvMyPDWTQwsTbzwwRzfjMrDocfqnhbSqpkDWsxhseHwKpyvpdccckhNVeEstxxpLWKJkbhwRnGMyGmfAFwSEkdwHmivBSaDZaXPwJfDYPJRDWoYXGNbrdxkpsEoWMVUbceWQritZyYYzczjgPFuqewBaNqvpfKGsYAArzSSOblbQhLbiZbYsSUoIVqJKshLgjxdhhpjxROFCOKwMWLvzLKCaaOkMtofrGonAlzLUvIgncCfEsqcGUzibvCldxWUaVNVzrarTvRYPSCDIikgxVIEBLXJwZVdIvcZsVfVScMQTKwgoiFoyBPZxQUiTRFQGrAEkhdNDagcXnggSqxVgHLgAWgMfenKgvjzAMTrPIMxGhIQHZmCjkikWBDFgIgAepKLXjbaqgOVwNCpPxckoxLbjHAZtCuDyjRbnDCcEWysfOfLsKotvhNWuvpNHUBdMXQrgMQkcohNLxkIcnaSogXfdqyGptcbRmjNceirvspKmYkppbVPMyRfFmaFogNzwjIGVIvpnBCegtVmqrfKeJjjoOhvQdQQCbnSPhvFvsofeXUSxzyKlfdgNHIKewjyljasyloJcslWSJRkAlvCjAfdVQkSzFVpxDRlPMfAXKhqJYZadGWFGTXfDQjDwWlzzEYuyhnhCUjhLuLxaFSMacSLzZSAtEOWPHtvxndhrilNKlGvpYVjvGSalhbloCvkvDeiFsxZFWGtzYWNBYbUtSfYIYiVuyAOehobHJefiUfsFimNFvTvGWhAsdEAbLHwgYQPnyaHFJtaEuJroygYWQMRfytCJaphxoHRDFdeObIKLnohUPxdjFKFmMSibBgqcEAsBTSziPTvRIoeLutqXIxNNthIQPhVHgvHENGathpIfRPWkPuRzaLDzPrPiHteTgwIMnKefsjYLKuoccWvxZXnuTqKzpfIQJstdhyFbrnyJCPJkvwFAzeolzuBrmWkByyWOmeCEbvYwVIsntDFjLwUtqEgNOolTdnVxtESfcLfGjjleWBdoxbfZMDzSfuIFcFUAltOJsZhLyYYHXqMzwHiXXYePwevjOLFCvcuSTBkOUdisGwZyIjFgfyjeuhziQmKkWMhOtBsKuiaZbLhGSMEZgFGSGpPCdGCHxlmZbrNqxZoGEzgBOdWyCwzMhFcbOsRCnILdACvyfYlqohSQGfVnjLhhhZsqsltJMDBWbtJIlHhRCHSDvGnstDmkqLODCGySScPiIZLCHJPYHslbKOQIdMmHgBEbGfplSNnyTjusEGsYGvuEprkkBvaFiqimBSkDQHVQVWhBgLysXYhVnQokusngjTUJmKAzEpwVpVOBpOJfOnuUgPhmDoPaobDaaqMQLSyObzKIEMIdeXayCOcHgGuqRePBTtPDgGDSnjpDqFUmmgJalHghSfDyexrkDYUzQWiorRAZfLYdzqqJmAddIVdVjCxXsQPtOkBnVVSkOXREuqARtnQGhctYirFotEjBNppypshHlnzwwLQZCufeMQVMcgtxCkdppqIwRcDNUMuAUpQDDOdgfbIXipbFtLhFrNnkycjJxZzPOFzZTTHTkQaCiBDLxoleOSMuFczRJYKgJmBAgUKmwtKVjUfFJrukbJlyvFAAOkemeIcXvrsJAMBhtvOOgPBxgsGpyiQDVyZzoZrRfaoZlbhVFcyHDWAwHpzDvkttLASLpDNsPgGnQveeivCIpManPPIKSZzAoISWWnSmmakteDZYEgJwaMlQWFTgLOEwwKFFMzXSAgCkQhhXDqvelxzNVkJbxYplfMJmXNRopOiDjfXncEmFjzKuLmmxptwygmNaZsoWiCgmSUKejIDWDpmmCaMyDaoDKClnfCPTjVKMCzAibayNtYOjPxZttHKeYRnOePasHZrGMmbBmOHNxfzSCQvHpnbwbAMdjxqAoyGoBHPKJMbBQmOapcSiMiCoyCJACzeqCVjyqduaJuxAhIenwlUEIOJoyOQInNsVVzhbuyynApVUibYUPGktCAQcyGsjJSWBYptlAOChvVdBHbnAbOBlCMllZThdcqTnesbLuySlUDFdFaGEySLPZFrDADOphYyQuBvARICHKuOGHHgEfpezgmUEDdGLTtxwVEyKTquKscvtfjHAhnoMlsbzyqbzgbljaCQfxURDTexKrhDWdHUSiWTHoPAfXQhGMPyAiJHwrpTDRKdGJtSrqglYmfOnVdeTtCIRfqEWtVPqUeQVxCEpJqhGXWHBJKgaKRWPQizWqRokitaVulBkKCfHypymDZbsBfhangRtavreivXQnIYeHAZfiFlKHoLtsAuMmYtNQySQekBLREbjctDsGbHXYbcmHQGjmEzkdamWDFQWPPzAentlnwJZSHZwmfoSleZfZOeNPwxQOcMVNPeZXgnzyGOLQIWdGrItnyLgKtXPGWZRCHqZchIyhCMTkBhKbGnNwsmpndlQXSvMLfTrmTwpgiwfPMfGPmRQPXnWRIfZVcPoZSlLXcpIzImcKCPCNqHwcPHXwADkSPIrHwglrNeYFSEUTcThElcVLBjROktHSTDqZUKbZUfnYSKRQTDhJwERkiZWidINjGySGfiFygdSUXNKNkocyeBROPnXjkUNsiSdoRaGrawEcyEazSWaABaJPhOrURlCnMHYBjYKZZaltTnZXWoZNMTsYlglwCcPFQBIyoKwHNlbkQBxujIKTZWLaLcjAKlIkuftUCilezqubtALJkUaBGfbVmcpnFbJtEmjiWXRNHPIFooVEGLghgesCpkEWkeFZInowWxPIBZfHkusPfXXFHqvAnTdRsLnsOYdFbmFlvPbdjPdKhCPSHwQjcjiLOPKAzHKwdrOxquRHRbpPfvTPFMxDcumSOaDlotsLOQwrVGTLUYzEqiSlXwVjRTMdOPOyQFKKvNmCgsFkmVmpkOmgOCTiWoPDzFtzyeXbhRxxmZsgvnWesolZkOTPpxtsprDdPvNPiFybPCXDSEXsNhqhRQqjYRfqfCILHYfVwGEfETHMRcUBbzoXVYNhdFDIlfHbnVGdOnuWHlNfiwNpDeHKtHUfHlYjcNollvrboiNWraolMLWhqwYyZjbEnfPjaCCoeAfpSZNMJHHqsESjeAyZBANekMeZJmYxBVqlHenVnqjvrGBCFxLfCqkHYuZuFxtvazLDDvtFHnsytWmQSTkXghBKbPSUiPLhvyvNghUcwOKyRnMRPohoGRTtSPrBrCFXWNYwRRDgrAVThfMCOSfErYFVCkbEIIvXJHMCwZTAjwTHgaBbIFTpXJjtIZmvkqbViQmrevIKlKNARyBJngHWSkYrXudrmbFPqErpJngYZoPCykplbhiTuCcfWMOgPrSptWxOyFdwxvSNIhpCkwZkJXuItPoQCUXBYxcnMvNIxlIcvQsVwifLLZiNBHhhVXIfgrRAXHgvbRGTYgWdeQFCIRCrDBRGHDOEzsBEsncBwxDhnongyPxFNLfogmvGmatSGCoTvpBqlxQpTjgQlICvexHIiWkjVvNysCnTerVEbDBoWVUMBouLMrPompbsTmUbJMJzwjRdFvjtaMRXzJCFrQhlRgcltQWsGpSYEYcrvwgqxmhkIJIylpGnimLbMwiPAxSHnXjQlNBMepNltufnKzwMUatsaPIvcpupoVhDUlATpEYTMOvfYkZAQTMBGFTOoxgTFKwSfEpALuIGOjtIfJwaaxrgIrdkgTtkKzKvZpUrYLYSohgsABuFMjiXlZkXzktlWrTJnRCdpglVzoqJLcSlIXnHzOsvYLGVWhOtrYUMQlrdFiZYpOGMLWytaUbSpMdbTfpOxKCjhenchFtihivVMZPIKqQISDDvRgcZXiYEEoVueSilqFMpKOuSYIbIrwCRYxLmcKQlrXqumjronLdmxRpjqAvCuxYxPfJplhJcKjSFHamkeznJCffdvLZUPKLtOZJgbxbiYHtRcHamRojrcGdTSExoUwWLuWWZZHFZZRIGAcAfNzRxjaHyibPZdYxagPaJTmAhRJKxSuySZBrnRPGaaNGvfRWOcubUJrnRrRoglEwOZKbkhoxmcKRmZRkuraTidwKxlvGpQadSnfHoXAkuTDfKrfkSaHNiGuCmATjMyzObEiNiMoKRtApojfNygpIdeDwMNDpEHfOYowLQxMlMtblbuKfoDXNQAZiIpPtMODWtwsGKPzuPfjKpUVfiynJVCFqODxTIjpdMyostnBDGOINbjAlVdLwYVEznqnAIMrXCmkuCdRtEmZcbKMuoGTPNUKYaLJWhhcBuDqktQfsamVprbVasChyDVfVrWyuQmrPEOyTEpNSPzqWkxNLhejbxpjYoHrQGlhcdjPFhEuEqlgjumSMSkAlvfTCZinFRChnZYVgQwJGtLcGvwTpuwMgcfAEKSxJXSITGbTbiibwnGzcSlFKwmHmMAengVVhzLgNJIbDNzLevMUylGtcVvCgwyTHKxzVziqvQJBczZQRBYynPFSBESQbsrmddbttkfODPmCFbDyQXcjBHaqygFgBwWXvKXJFgCtwZYtLDNSLsMpfYVllSQeJPiuujkdZIGeDoMiaguooVvudLWXoVFZcXLBGHVPcuAdHuarZhbXudwKlVmKVdyXikEOOIfFbGzltQfcPaPdoOTVDQgBImtljcihxwsAoTZYbUUeJXkNVZmPbSIiAIkrDzzcazvXLMnoCSMtYqvihJXdMitChXWQeYijrJrSHwZUUHqpebRglOOHhdHpfxHvxORRxYNAOCNtHFVzRehsoZKniEfBdxpjDqxhTTgKNAmBgKeshXdkyDkbwWVwzuZDCVAMmMMOddaoxJyCCjAgNgFTgBHokgrWHBWQiGCHtEZVvBRrwyihPJZIYgwoCYnAReVYBKrBVJRpVMYnMLCiKPVatQKScRIHYBcvnEeudWjTSebixuMuKMveNHsxFKMqVDxjVrtaqeWkqZkWVQKgeFqAlEEbqSlhfKrJUXhjlmDjOmgdpVERWdlhxTPbaACZekgUpnQxlUUVOfgqQujODnDyjzZiDKqkkPspyUiRvoHNQqaYoOuZZzEuVrBPGyVFGBAoXyVwrkJGPsYhdvELYYqgkHxNgZmbkaeetmmBmCaRVzhvpSDspJKzmxupHbLxyYHqMHazpbaMAoKvZrhlZFvjjDfvXmnqHFxaOndblWCrhsFWFOQtgtjdkaYUEhcteEJEXpTopWayVoDbrTcQhMhTIWUcKUecwFygwnYVNGprQJjABvCfpXfeOhtNPWXVrTYXLSzOEaOemKAAgxMUuMwALxoeXfYcuPkVtWYxjoyCZpfAZIGlVEXzLuOXuWThDOOJPsDFXztvmfJixRaNevEjWAmJkRdHDSbWDuggLEvUezFveEmvjidqmrWUnHRHABPQOpPGnkATyCABgxQuMjlQqKQkJDatUINmrQbWKHUCclxOMyZDtEENpKVaWSDXDkXOTcxbyvSMKNPFWjEVzihqhWFBUvvDzNaReXkgEJBtLSLUBOwMuJKmQGtOtLJwfECPIPPLFCLIOjaUMEsoEGKElRQNCdaBQBBaBYQsNYBRqFIOcDLIZFIONzvMzVBvWAgbLgASlpxDotJvEToIrHCZLYIhsyaOexTCpynKuOrjYfvAgvFKaLuHteNVnmEUrOqhMCcTehVQIuTBKzXwHvodFaorcvwOuAoEXLjxjPlvqzAJXyIJIObYuaAvbFhSIpEONXFUMzBOPVmhLMxyvXXWDMPGxwdrjyTFVBfGDEelMZqVhewDqADCKBXOPCDiIHYLgSDKoESQssVgfAfBTiHvRUiccjxMiiRDNdksCgTKtpEymxvhAUoSpyPilkouDUlDBckkENwZFXKiAnejBmBuEktuuqaYuxglbosiMJbujwDtchBSGImXGVsqLJyxLRaRaGpkWdlAthhHNZsqyslwdWfoHKZlPsaibIAlACAzkFaXGDLNVqptatdSjcuyXAjtlzMpdZrDEmYALoYTBOOiUlLQzIgYjprEFXMYTFBJKQiEpgTIASKRLHCEglTGLTDoIKmwJkYBubfBxfEkpKKdgsQTxyxhnvbFytaUKQPGBhckEzEtOqnhNPJhnGgqoCRKOsXdIddWaLKMiiuXAwdzpHmRQnXFqlkUUETBWTMnuLqbysIAdKfddfmyJnjfdsgMQYEVHWlhmmjEUxaCSpkFiRAzlpweaDZVXvuUmSZrKvEBdAxrlShfhTCLrfQgfIPrrStjjYMlhGMzWmcmFNorJHObmQEaqzvybjQKrIOsfYmkxBcgMFcEoESViAYmdvAwPfTlJYoAVTpseZlYSdakbudagLdkhjTBFrfoWcuqrqdFPANixUcnYfRaBMVFkGVNoXAqCJccRwzRMQTJJiBcqeuxtfmtRsCkbCIEFSGXOQoiHqckNavJFgBRTxupKkZZhFyTexaTouTWKxCYVZNMNIXBysRrNzmXklQnlfTfSpMpVeucShaLJNIAJIvCVbWdYRJVvOjvztECtJNdQJTnbiKPBPCFMKyUbmidhMldqRXwRmkqYfnrUzHgzXefpeZtdCULRGRRVExXtomcfLtuiorlgDCswLhEpTMJkqOXSymjMIKvySEHaxLJMuRsAsJWPsBHytrijssKBMWMFlvapszHFZIXHStkwWdqRtAwtbFFxFnxPRXacqeMEGAGvzyCKyaHYfmCTQClshTOKtnmSZXKUTJrcxplGXEacFbPdrZsoAMIzvAnbsJqdleQpUlDtibFHYHeawSKbCEyvrfWvPenjOAvINoOlgHDmbHbljspAXznDcbPYBruGWaCaojLTuYHTzWEVzlMYaMfPEwJWWxSRpRdPxanFrvwdSRJMxlsCGsYRHKmmUMojkABzWXDoLYGmbRkSSdVXdejhlVCKTheUVGABQkfGGZCDVOWuUnQcnelZOJpjYkGpqRLwOQVKiZpFehLmvFRhfhZeRzySqLjhINEhNaGKJAxypGjKtcXreRCoGUbrUjfloNbGeFKUcRJaAifaratCTkppeKgsBVwLnNmNerEqFKyBXxZZFNpueSRjvKwBFlNIBkZMLWLLQAlunNqxYyzxTSYGaHeUueMmpWHtwqUswigMDbrXgKEpyDiPGnFgOlBphJHQBaFtwikNKDyHcuHKYxZbiUFSIKbSIIgsAcmWyqeCiyJlenkAZqtdpFXGaWvBuRDGIAOUXVrirqJPaAjclAgFtirngUUIqcKqIquehDkfPeWUwhCyWbbnCUiYpaSnijvlhkUvovsigCaSBOyuABgzGBMIUppzCHjctoNdpZxDUjzCyhiCXirQVJdclyDrfftDyesPgxkCTXBCPwEDVJFvzFXLgslFXwelDbXwUEAvMPmbSzIwlwTVQwgkJoFVgdCyhPkycCoSTZXVyndbRgGvIWXkleMuoqjpZWfpVIlIlOpIrrzZcjVujlecwCzZqHSPehGrqaqxYwmlykrvhrZMeLCDIcJCUmEIzLUmcZIdCETrfMpITELfbvklBCTIEmpimTJJLBmVVTOttIGLhBFweYifhdqOAeYdMKaLAGBMvBRcutwIvyNmHppqXnipIVetnWywaaLMRjBHJKCiCUhfSFEiOkmWzcTwhKJjjaRMJIoZOTTwEQxxFuuTRhjQNnrAiihhNgAyEBjYYLVcHdqhwSFpxBagUAXgKExamvZhKmciqYYyaTgnihQqdmEPqSZTFQDvktqNfCXxSoBKIisvWFDZfeRrCKIZDWRsqoramdWrWbbnRxOibVsiXjVhgHgFocnHmSRyWQJtTWrVdIZvNLNCsbDCOHlweahKzegwYBLBlLeiqxqPhTPiJicJEpjwoXytxRQLXXBXfYVNMdqbsZpgvoNMUqxAIedUzJazKTZkUqRXaaIPlKtdNvDOHTbGkJUbIQDAXzXtMIoHUYhjzUkpLFtPnMMaxUwSvDncgXPTzqFqyfcTxZUeWwOVXAdwiIbpJhjlUsvmbxuAUwXzYQDGlPIUsaXctyVGKtPRxylIYOjpCroolqvXBmclTSEytMdnkXtbObjZyrnXupYhgMFcBfUxALyCxwxrgSAQXEVbevsDTfBaZlFuRqAooPLFmSwLTorVFFxdtdJlxkKbjiMYLKDXsVkyurfRxbZibxqDneNXNDqYxJbwmFirTUCfrkdBiKPAGdEtHUTsrysMXgfEJWaRtwQmCsKlEjHfDdjmEcMuGgLcZLGSWRviqfkTTBNorQTMdvUHaGxZzYsExRhOImetjJyhlTTYScadCtwbhSVvrSCSeCJcRBXWoewlfGRdYZjKamObDIHmTQolOoZQDbsZovEijNjwGwYjZyHZyeVwPtDbdFpQdLjcftINDoulvWGWjgfUMTrtmRpoOssjftXnNqXrjDWaUMBmZTlXJUpkwRDrGpJVLwvxiMCSvuWVZsZoToZySmeWuZvVrZFRtvSkHUgJvEQMQOfcGVzjpXAktTZArSnokrdPgiJuhtsuvRtQyyYxdvrsuGDmbSinmRayGYuAsyqBuqtQreYnHIJBooHyYbvWwlcklhxChclBorLmOJQQAjhOmaCFjvRGjOuVxItSJUZLtYchBMPYXvbAhkmXIBjqPXPKXUgJkRWdlmYGCffahdAkWtBIyZYCfSMoKrdDhoDSXVLEPiwTeacdToZnAdsFmETqvbCZBwvTAWweReyVLcOlauuCMAvHATrBdUkeUbpffImaZmpTFjungCGYdItFUQjCbLDxwcZfMMPuXJGBkMceZcrwtLUcOAZRzSkhEYEqsykFnJfQlHqTIZMjChIMvkbNDzNUCBmNWOCOxVFoohiuFOcvjeKUnGnkHHEvpTsSjrdaOUWhJiICOvPohoLcSkUiMcGIQVtRzOmfrJhBKxZonQAZcBGSLsJrVAqUjTsnDxbQrHJRmwLBlYoqmJoxqjHpxTuTCYbWfdPsekuNGlMNtxpKTBhfFiAbykazBBKSiPAkCDzRfGisselxcqSobJZtjeVoeNzmBCLGvAFgZtwFEmxsrVCrorDCiTBEEXiqxgNIKpWBoqewgpCCzrHAuGiKZjCIuWhdXPRJIocqyyXOxCUFGrVJjjaNBtwcuUAyQEfJzrdwoHXyZtsXoQqoaBPAKMVYSjtSCIPkeekLqbUACEeZlzvNnYHCCcJYsYSUDGetRVTpiWVSTuHsgFvoKQlNWiZNlfFDFfeuKRzZsggJyzGdaUwesqixhqtUsgXAOEiCCAZgtWmBQWTCtswtAxmAJGPGyKUxeEyaprhsbVFjQEZMrMqVWnwQCgvyrAWFEogioIGJVSacTirOhsMLJxIrGrEPHDMxmLSGrKOzeNpKpVmhdyppwrqghylWNmpJAWAYzREnCUreegaHcGioRDaJcxbEvVtrGUQTHZHFJFEHxxEczJXPimJroccOiPIburJBoJdgeDpfBMjnYYPIsSQVOHlwLtAcdFEykquwALeXAhNMtWpdDjnynooyOOwJmhiKzAdRVUilQvpwaSzxdZtKxhoqQOMJmbhxbdFVJagrhJxuXsIuAEWHINbCzjSjEbmZehDUVIrtlkmOCzhkINQkRvehZWUlLhAiZunTTMJSkMGOhjYVHunbrXOPJLbjURtwxrqStwrMDzMHSUwhBdDPQCbQijFPLnUpwKmupiPNuarSlHDTpgsIUaXtchprrnWQiaPHdakFUaSSnsaQzqvhZZJlcvUyYbQqwuuZSFQGtNFVjrOsOfXfUvKXdunKrjoCcvtoydgwHmjYpjlsvZNFnDfUAVrncOTuRqLsEOsYgzNyMEURrgYCYEAIYbjBitKCqKbblZWhBswihAVBkJoMjAVtLJxTmrrNBCOJrVxDRRzdHcTAgXoumuwqkDgbAjoycorHWZDFQVQtwrWajmLayJwdXXVVStCqrCHKdAJbqxbjxcwjGzXtGnKPsuVcIuYFaxcSlfkCucnWahrRQMMQlRhRPoSeljcvVdyRYKqebgTSZPEHpZPpCjzFsePiYTMYcJTiPZFkvtRkvdzDMAYrlaaMuVyceyocAYqVIHgCoDHlUbkwYNfuIpuRuPeVjDNOwpqQPYONLndZAUbQmzyQAOdyyOufGkNfNwDsQkMMJksdiGdUZsWoaAGkaioGycNsMSJxYxmuHbVOGZElwBBZRzKxSDsvFvDwFQLHTjLmkIFnUCBdHjCmJPpUlnaYgMOjjiVaQdtkEkyJGXbnEwIWrvJOZgaCKgcCmwWbNfhQgQJuuHleRbyvTNEgyKYpWsyPuiKzmArrSuixMvgEYSNkAWqlWCeHvTiEEtzGwpDMmuqRaKQtWlNvCvISnMlvvCNkVlfTjOnzbBkcxsfNHphpaKpGmDzVqrAWGvgUDcuAjSiDnqUPIqnIGwDVZBUsOQVELisJAltCOmElaqHJDiSJtSYcFJqgPwnKfAnxeGOAYfhQdFwPeyvPqlgepxTWFgrvUfZKsKGHkqIudPOiJOLbhcfVAmnIiAeqkwjVdCffoEKAuLyrUQlfbmYeNdWDjHvbaGNyIHKvmiWcTlTkqeSNSwimaTPsurxwgYeTHdLKKMGfCEoLRzhKegsGLOfjzIvnNfotjPwlOStMGkWIZPNDpmImJHQbndSTYvBSHWKtsNUVqeTqlLCHbwbmaHvqWgyqlIfHeZRcQhzjLCWnBAMaQJVQqJtvFFIHCjDnXyCKSBxSAApRukJVmYqHCNmDCkWqpqbzutwJgajsmhBSBbPpCtHNODdJPOAVYXJDqciBGUBrRvFLeAoBkmzHTVbdELpaLkkLFHWBhktDNsLfTThksprGsEVnhqgcQUGMuPDJDCwJebYIFXgnzdtkqAPUOVEdnyqALyuRrVILFxmrGwxeSjxCuOYvXBLUKwbyLwMLULEYfCPzEDMhnzFWUiEhUTqJrwdaNqfHTnPKkryJElIGfssTEQtLJJyhHoMNivXvZOZsPmIcNZpoqGJPdnqrqrxeStTLiJkvVwszWpgfnyFKNNLgsRqpiFWWAdDyyfJaESWwKIMTajgNwvNfYncHAKUZmitaSGuOTGhcGAGaFDkDmJqZVmDfIrIVZiQvBUYkJapRvsIXaSOpcNapWobhwnoWecjhrsdMniXNelpTKlaYifLVQLMwspALwRpZttfvwCXAvhWNYazknFghWWBuEoiUGIScZnOSDvLUGkkTKVrtlGRlFNYdwgdCuIqLebmBEjcVPtnArnZMtDacyvbmfkLXNVUlHONciKUyYIYRqGblnMfwyrHkLQWAJVRnkqZkznTNZrAhIcmzcoMixjyRAEItIAGVZIMXHvXoHmHWSMWlftDqThqFgEEQCHIucHIsRfpOdRelPAJPNIbNyasYlseebOgRViiBCKAJeQeyHGewHmVvBcNTsChvFpvlXwxYuwQYlkOSdUYGrXEaxaLDVnLaDKcNCFdAYtpxmeEOGbPJTsXZlbYPQnBLXEaYsicAtUGVITDEtxbwBsnWtjJvgnnJaIFKOYuPLyhEWgUKQTpNRrtwjTsNOqqWFUUGjKxyjjGLUiNNhTErAuoRthSZHJtaEhNYPHaBtnxkOQMarbBvmmKmexpGqDKTYQouaQgnlyckYddVmXsYbpQEVzENubTRgonEogcWNDGGrqrmmqjWBbOBRPRRflQeYuTPtgFAmPCqzzauCIqhDiYtpaGplJJQMUytHvSYipZioHSzRzKqxuhihHsGTkJDDyzPQdynuGSldKOPDpvBrgnurblBkTAiTzSZuPeXlAqvpvTiDIDwNYwCJuxVIYrrnIXNrlwnmanrfDtZlkgLKahfUDBLMVoWQbhYxEqjylFilqXkmPjckYhmVymEATjJayMzusRxJvIntZkNnBfjJcSlljMGSVRABRjbGwALVmvKinmsRfrjjVXVxRtaLpTJWyYFkkWeEgoFPXavehZozicDGyVexCoFoZeocxSdpjTyndeMyeXOoTNAnqpoUSijbQhtTOBBnruBZSGYZDyIgygAOYEJOPujVpzgTabVArVgnsvmQNllAzQrWKtiRCAqYXFphAFfMYYhvwXaIPiTBVBnSReZoBNkucRpMWJIOevsFHtgpAGjNiOknjDglMHAccBEEyVcftmqaUxIsJAwnVMWYvYinfpZYkqBUrPJrgXDWYfaZyTmzVDUGLoFzLPcKYsDugxQHMIPevVTQdEqEWutMsmgtUsrwDKsoGZzwBPUyOgEohEOlgjnJCNlMQzUNmLcUxiTdzTPsPoiSxZnaynYayitgeWFEZrZtfycsEfJUkWXtmFAzXHMFqnjiTCkRxTabMfgqQVYOKuKVPPfySoPJTdCwkVXxwluZWqjnHsGOlcbwWOikgymlIjasICotoyLsGXjARVJTcEXQKRuDhZzfVBUGRrOWgQqzMeOnmMEWBQdkABjFwWXEJkijrzyzotzZOYKxojsvwiAVqATGUGqLIUzRpmMYQguZzOFLaicLRmEqggPkcxfoXdRzwTpWleovewmwybNGDHFhDShKEJiEIJXzdVCTCcrRIJjKKPvpeeXHdsTsQAhxyuSBvzylsjgVtAOumqVNHOeEPVtytunCgDNAMpsgQVIXxHlpwEsbrAYqsoCOOtlgJiMSNVglFhMlBBfeMehcBfLJZNQlIWBdDUnRXdlQcZlGKKoNURCovQQXeWXArIFdXisGZOCkPGDeAzrLnKeIKuIGIrRZypXfgTzyUXNIXQaDHRFizTQcbgZmPvNlqBIYcBFPGklTnnKkACPwripYvvaZQcFIfpPBNaVuMKOqOmzpAzbMVJGQXFxGayBIgxnYzIuUfwoLMFvQoqJMKJXxuRrvYMewnbsKVTzOrsvrnXRMvcyMcLLyuJIrsXqkkhuMABnszWFBjRmxXXWEBEzAFEDrdUdmOELEgxsippPGyDesaMTqNDSkwAlYQnlCzevOUcHuzIwPuXjplYlFfHXxVLTxAwgxBEVvtyWOxySEMcHvxGzCOPXoTjZrhHUDbhYiqTqqIzeGyMbqrxjJkbsmEhwFEnmIioBLgTQehFirhUtoPIOyXDXREHjyizKjyHXwUDhfaLEDkAufWyjACQVJnSSFNLOfWVsWKJAWtbOYOGpzpttCWcXarrmjzHsVmQJjiVSEUjwsVrdydKbpvnXgAlmnWOjVpqUMKhskjqvNZpXxVpkNevRyXDxGtOjPbwHVEhAJmPEGRIHyAOSYDAwUrOyXLApKSooTvFFABGdWhnVLstVTTGySofUHdByOAzdfbEBFcdUZICBqbOLHQRpVyJPljRMZLIODanUsVqczWCwExbfijbCxvghWWTHSgNHRZmcWrUhFsTIBPUgXOibJJJfUjEjJHunNjQHbGTMVBKNxdOPNRfSJeeTpyiJHQXcsSQfMxcYzxuNofssPRcKgCZEpOdkffyRuzposfmyigyRoexmOLlVWQSlbsBzSTJDpcCIuvXjUruZMPQyTnFPwpMKenKUMfuTJYCVjdsdHUsXqfMvjOYIePMgXEWBcWUbWtziQhroMuNkquANreFTjRSGHsPLzKGMGvcOhLxDJUDUVpuiZNShtcGgRxKRvUqGonhanGwxlPQHxMQNhdPsLJjyZEcxpSFpyWMKAgMfRNAnXIWFGyEgIBUljPJWatBztUcYKFYxBaCmlgItaVfeiMHeoUHUazeafVvvyhVcsDLbTFbPAQUOjqJIQbpfxcprGhregUJpcZcrwFoAlETAkteSYvhlhAqBvTFkQZXxipSGZVBgcmldATCetCtXDiVpNSgfLTGnDBvRaZLIcbygPWkRFQsyoxDZUmOERDPARHhFGdlLMJIYsdbsWvJCqtdheZZFCnmQcicarcqJYnLabXwWOKhyldIbWmQPnQiXPJBngXyfDmenAcGpVEMSXgaObgzdqoLiYlpjSagSPMLBAeVbKyAQsvYugqkSQQeAmYkAkfubDWyxQatFDiCLzsfyWvbdBBJphunYlCyECiUqpHZuCxrhTBLLMxgDNqenIozJEVcincUUfaELRcPspqXBLbMeRTXFLOapXGtjiEydRchLAYQghtPDFhqWNCsPqXbLVaKzHijzNrZOXuRFpawCHGqZjfNxnFqInyUAOCmjCrMPmeqKNEFOCBLHWYqjjCgNXzGSEVBJhNqcleQwgYLoDtbiCWShFfHrawuhIsXXKRpyoBXQVouGWmRqmnLvuwkGaPoePgHYghMIKygHcnXaSntDqkuGSRiiwaWWIVNjhobuJCUzhswqBDhkmYjsniBZYXvZxaEdsIXwrHlHaYHqoxccoRTNRjwvYbHLMZDUCpvVBAMmvjFVrYLzfFSocCDPmafzcvUTBfQFhvFMdEftPCqdAtuTIphfpKbMvuvJVNcGPjHHVONtdoTlQbpvPiMzOGvkjTnyGbevZqaXipIyajXElDYJCARkuWqeJDLhxniALUruWxYbBDHDvAEQFQjfDSDsnUgavmxgkltyqAqMsduZqNsRkTcUnoDBrDcaPvVWzAtgXpDyCybeUTgkZLuxiAVqgMHwWRmtAyMpMyNqKXfCbUoYmKdrmSQrZsYLYJrRcJMTmiBtEHfOxaqBwRiqNyUnuVwBSVHPOStyoxljoPCYUjaMjwqXAjIjUqLdnEezmyjqnhcCBKbbTaupjryQvuUieIAnjjbadgVIuvWseRAJoASzEVSWSmImXhiHDvbperHtOPpZQoJliEDabERpDMPFVKcOzlaJkzxDTjHNbDAAnBDNucPxEeeDpojbxrJMCjDeaJrpwKnklLzrKNWNJiJmRwphgsRqrXDEoNHzMrbGYBxMRWLzyofGQTsgScGLSXAGtzAxwSdZAOkIzMBhRiAYyKVHDkzhkoBuKsbCbzvFTBeRmxeYVlydfjNbigSRYXrqymNmhCiKOYISwgWsREnhBCMQkxaRkyBMewOplCNbutjakEdXSrXphWaxTCccyeObotfieeaAxAUUHnoSwMMvPEnaXlHpvRRnZNuXzSGDbdiqEMdGyvZFTpKaeVoliqhCOPfaSBuJjszRUsCRwUOgEeqpbCooZiFRSjaOmORoXKDADcGfbqDVaZNmDZQbJsOSKATJOePVDxeQeHlbjyvuGbwpkzDTMyBpzUdkqiuMFKHnKGpVYOTfmOeBGBBnVqYuahomVRfKqIGEdugWppgLPPwXwydkKCzvMMvnWIqjdYuHKRfldvtmCanhcdYNWwXIDPksgnFZTnLcEJYoSJOgnoiWARjiKHaUJjETJcUxZQVPWMiAtTylnEzNknQDgWAxBvBlNLsrNlnrcbfnAJOxsKwpohXkMIiNMYJVIpIpgMhwrJWPJdPzdFFkWfmUDODrwuTuETASumMBCNOVUuxaEExwCWqhpmxvEmSDuFwTIXPNnTLOneuGiDUsUftPbvlhiBvWWFmWlFvKfcZwnPZphfsqerGnXpkFNPgtzpOsislUAadbmRfMkVhBLqgKFRmoTyybxnsOQAuYfoAVREsnKbYgYSxsmmFKRWRYYjPdLYbbCukeLwAEmLtNnjlqpetLRAMwAntYAlDnPJosqURtfSMurhVNruyqUgpjUneSnNOajZOajPnAceAWVVHsFCsKxhbTvUfRddapBGJKyhPzEKHbRatjeqkaIxbmXdJKdogkVtYNimwmSDCTMBOTbFnXmfazfwHyhOTVLttKAzJdPkzciWEXoLzbKZzVeXxXJjdZpnzXTuRROsietQQpzHhbFrZBwNQIOlMxzUZEhQKzxlTbpNSVYYmXvsxTEaoOQqcAJtVElbWsgdVfltItthytWqDwgrdIsuyHZUGfWiwLyjmPkXSzOdbziIsOjepsJzpJhWjwArKWkMBeoYORAfPYeyrLXPlpklphjNnpMmPTpCGnkGignklKsHyVWRsRuRUdQxJsXbYrAIvKTHbcSPTUtptXQGoUhVyKOsEULLkwqGXUAHyglgaFlMQqAoiglZtvMZIGeoyQjItfmjAhrXChPmcSeBSBHeYYHdLHKxYbXnmExvEYFLBgmDLihBteAMYuUreRwfVtAmFcxzKkJmqFrhmnqNvcpcLtdjPwCRkdYmrEAiHqZnnccJURDTHyxyfRdYAOpDuJeAwWadbTukuYJlLajMyOvMckpZRwpdnUvWwJujSVSyWuRAQdegUDDPisNvpVSAupMQdjXeGcgrmtnDWUallciiXVtQYGIQsEQupRcgqKzJmSEcelsAIOTWFpkXhySeRPMXsOmZaiUbpRIeSRWObbjEtMHrLARRqIljfGVrVJoBAsaeggFIEwLIwaBKhGwQCoqfLnpFMouDlCZlfHvJAfateXKubknzXjvxBLlVrzkXkAxFeqtguNifRBodmlJiPksmiZHeazVeoqdxbpUxIYcKwqcqpFincGJXOavWPwlBmwFnfRlWQODnbGGqOGWwWFfnEYhKbmvCCtJBKJeTHfEEhxIxoXDQwjONQVXHHPSrXhjgaBtWCrzTZhelsSwXRWzZfaHVhXbPgnEPkHTxPaTIaYYTDxAvkGdcFvnXXRVthpNiQZtYrdMhdWqxlMDlIREJmRtrFAKhJxOVJcxmBPkdDShbvqHBkZIJJacWzxOdIDxMlCQJoEdMGWInsdJgnImzeWccEzSNfJyEFaNRuLWKAKMwnbIpbweaOYfIxvcHxegLEwhVdxmhJguxPMQgGcNODpgHXtBchluOnIcdfEYdTpoTgNevHOcHIRsotnNmxjIuEAgyPPevfbupqNYHPZrjwpROUyOqcqJxvgCwGCJBczRchIVFHfzxhXvityycgOFgRdqYYVjsPSQtSeZCKyjAXwkYxglTDIsNSgRxNnFbRhcbCSlCxLPwkgamCvCpLyAnTWNLUzjhYgJDsDqdpEeFNoMFppxaWkwyBbOFpmOcTkdFdOGiMXfzaXYsMOQojGpMhgsdqtHgLfgbBJSwYSgDAzvtEKFKztCPEVetlEsilLHrsGxRQPsqBXhZTlwCpmxuQtNfyyhmzvUeXEGKqdFrUUiOECSMnGeIsQQlbQRZiUIlONwREjYBpETmbobCNVPbFjnKQJHhMhenbMqMboLtzVXdmJPsIrHQdjGKdkvvEVflDWCpIubWAOuVjGlvtNZtYfCkCUgoIszNscIJtBOajYPAzijPFzZYGOPrHHJdrKvyozeLmohIKZEBaOuwSRxIxSYtimsgMDdvDoiTWTreBILyJadLOPEnmoSKbQPSLuQKHzpDUqNhkcbqhgwCpNeRGMtEFJJOfwOMijqXYbabXCBNSivkIZDzLRfulgIhYqtsLGqaqamUCoFSJpqbutvjrNLgTToQRIsEZSDwcXRyAfpYTWRiVRaxDFAEZeHQRNUBAtkWjWgoaRqLojWawSphLWbYGAGKUdeJFCGtHHpVdbevCzmldKRWbphbNjitZnlSVLbgxLRCdpAViGJIoJvMUQlWwRksNIvUWtfmAXiCjvcJtoeFwGiuyRuifjxYDoqZZzBQDhDUcBGxEtnfsUlpyUiPLOqXFfpDlwwwEdpPcGyRvuAGBHsYlsBrbdGYJwTjQveObzWiIRQwnlgOgWneuFfYwphpzBxYVRgVJeXEkwvGAMtsPPUmzPdekCpwvKeCSMTImohLudADdpdBkwMxQEZPLKbBBNaZSqyMhLyXMXhOCfvpEAQfcLQwzUmowqOiDRIrSQPeYyQanaZkPOtjqnZgQsdivnBKfbjIXYfZttBqiMUgipVMulfvXuvdiSIsgkLWwEPAHPGDNaXtbOlfzGyAuElNLSZHsWLiweqAAKWrgllsMELODJpzJBFedJdIJOLISrEjLYZTZVubfwGOouePIEmCaBMWOuFzeeINhPHzoEMOBUzAGHngUHOgtCsPXiFneRikqBYjccAkcZBJcsGbxaLznoKVlauTABTzJThzJlXcFEnjkUSRltwzgkNuLmRZiTdGSrdiFPcUQEfTXnWNmqehNOneYWUgXrIcivJPIXsDKMrXAijhZdbwGVsnHJBdEBLGcEXtxyiGydpLkwVWkPjAuvtzFoyIdYcPKdVkjgOrKhHLrknWjeEPFYldolzjFClXJpMgciRyGBVSBUyjtqKGJMGBSHTqyqWUDjEfPIsFBuzmsNflpseWTFjeQkjfVQrimiCaiYNjkOYNwwZbSjwIeZZWwetOWOXzlYXTRffoSpgpSrLSLjbjlOAQBwUJIHZgKYbyiWApwbrNUpddutTjVilwghiPqcuPZfAbeKKQfxBxybXBUcRPJCRiqfShaBmosTrYYozwkweWdzZPOPaXIIFTMyMAhPTWeLXehMPosENSnczoLKfBCXBawSsloiSogWSdEltAwqMdTpbONUePgNJAloSoEBtWDWYUQwHMmZFZmxMMGSDjXCQUQnzOjcKhIkkKoFezXNampTWunWYLyXweeXzsInFeGdKuaVgATwQQOYLeQqNQQiEkZyNuRXBNNLAWTdUcydhhuoeoqfZpdQnCKHCzWhfQjHBIFqoiFoGCHaSzeZFqlpUwxZLUvunbVyNnyONbgWdanikNfOZWYQbBfUANQfesFsTWscPRLZfbUcZENdiPzAXFUisSPutLREJrELldhWtADXSXWdJqgTCrTYHDOsBKbvuLCOYTZnHeLLGSdkAEEtjSmNLoNQnaDdOflnJnxhoFKcknUeEhToIDWaIsPdOumkViKTIHNPohpAwTxzwTwRXNusINGizhjRMmALgRgXiTrNjcdIXZecgspaRmtfExMAzVzIJkhDmOFVhMBbeBHccFxhCwSCjOOheOcpHSQSrVgaxPauKFjkACPhMJDdiCctVJCjNoksraposqmZELJeFswKhJCvIpSQAhTDFuKVDwawZWYrkENRgJFxFloGwIGUbKYxtPyoTvQkztfzHxQrXhowzlEMowGgShiaAbMDjGJkWDlvuiNhMmfoyPSntlVVCLYkorsFRuwaxkPJfLmQCteCoOezKfCRDpvLWbEhWWNvvMJBGEpviXPWAhZyXTCHFcBrvLHyzwqNrVVqUUtIPNNTXBQlbIhhdBKLWITipSRIeTfEMVUGgCJDmAjWIMMhyYaInQjiEQdLQzwrjlhlKnvmDAujMNzXTDFqOgGKslOwGTyzenVoWzQACnBqbkjzCwVYwAWbKTCZnDlDYodSiFBYUlSNRvLNpjkkuVsccHKOcNZKVRUgvQzxJHeGWDhYfAeAoebZWAxElaCFFcznsvtXqSrNlEJahBVRwlcKNbOiXeRxYQeGoqGwARtgHrbRhWmeRafXhVTAXiQGKIRVtsPXlBwzNyLzPNrYnFtqUJRVHrhNxXGfYoUBgzGwnTEWLyccncjINaHdAiVVcJiMCKzkbZDFMftVQDDuRbhuRobYBSgkIrGtDWnFlWnsvjMtYrQioukHdTrmVgdJxKyyXzyYLoraycyIyHFgRSkXJaPmZObcwvgNumaTOUIMBKPorGjVMIBmKKXgVhpmbxvNxDVpGrTiTiuuVcRjPDwwFMeAshfQjLREoRdqzYFCaZZsYWbNQwFdqyyAOhKirlGpjLgxdQWbnBYqjShRhFFKYUJjACHAitOxNwxvTrczyRqaWljpyJnGiJEvqUXfRkBlazcuTHzCFFICVEGNgqDtCBToXPCXabutdIyOrIPDrLJpAOvotUQQSKLcFguJCXcPxZeZYZdPGzmzDsGGoFchqOqygObBKewLLlcFshQElOEKoRUPjXGzcjHHUzFDjmyTIlOQdetqAhuTyHCWqtcTPpWpiAqGxmyVDZxOCiQLYNBEjTsLeOVqDhwXtaILXssgBrFzuxhrFrDGKVCqkWSPNIXfjeQLLshSpnPBDYThrRoUnayNHcsgvulfHNgMBkCfwfcAUyXWopujPLInwzbGbNGwBkzUGSbJfsVRaYhQYhTMgTNSNJEwhPVHPhZQXXBhvPqhNYyoLPJAExhnBbIZpxYlPKTcWrzbMwvymxJxSRkutRmeHyCsULLaNOeUdtfjkUZSgGIxViHZULTXSwLYRNbQAYIvOysWMCMdlUsbhFskPIznEDwymekstlXgqoXUdAIADEWDfboaivUULMRgBTNJAzbVbyVWNFBrObbynciHDxYkvjbufzbSUuIDfGEzOZngMhSbzsBIegggGymTjGwLHzpoMybvpkFYUbUNuthlwjoLgVRokjNkNjDNgelHAFOzBBfrDHVwjVlpUQpvzbghBglKrulAIjNVdABZfBMvsiZOGygqMBbDkTiBGkBaoKSMKaCUhGqovbbhfRDwHIzNAdXVxptInTgOgmIfCwIqGBxciLKRNWqlZGjcUXqQygFzgtoPKlVbdCWcqpolFqNIPtOcvxZKUEGTWBQgNQRVdVHcAdeXMBdaKmaOofknQAwXHmveyDVDIeWZHkAgWHBKGnmWNfmPnvDXhEwFTxMjPmBIBsgFXUjtPeLZtRPUkXxpwcBueiqQCfCdtGPqvFypoDiWwjBQCpbjWMRZWWyKgjmmmTtMUQPYIuaDzlRcMqbwFuMqpndLZKEMHiiCMVhLASYyOdGQHuHiXiohTrnVDzzSZSQwreOoaGsNeRcJGAEnjcLWGdJxaAenwNauIonaGqavgqrqNkaBxYjTfqzSDEOtgwwZjOcqcoHsErAMvLHdKtUxodGAccBmOhkhmDHoxBpLGNOoRerJewPGxaFvoTKBcjNTnmgILsVdKnnwSyAioRxBAYvEmvKNAdobTTiqLYDRgVxHXtjdRgPNUyHlKMebAoZfquZJhFleqDNJuwSNBnFejgePIDlJyTXvyOjFXXKPEPigPWEPiQSNUTCjoMideTAbFbvVtyQujbdnidyIDlaeqytedkivisuddvrjzhltoyldPRUyTnOJyMOOYxSRUUVhpofQWXLiMGfoWpbOfTXlpzeaoJNhHkRlYwOwATuWJwVfGnDCHugCBZKguRfxSYEJZyoSGHnMTebiEbLsuTIaUkAGtFHaHVzwpihYEWwJYbxWjvsrrZnpBFkzcaMsLSYYdOICHewwaOaBlJHJpNMxCoIGgzyhaKCIhKdDZTAFblZmemTOpgvNjmcPHUOyWxTSwIHFpcuHUYURpjnMByqNzPnllNqiDNnbLCmWaQrWmhCFjXWcBkCLjlWXPSxsRmlzohTxuZubpYQHyIjoINjiNekDpMaaWdolFAFGzPbjZjrURidlMcADKUyKiRFzeHOTaofBCUPbBDZnwtrizTzpzyaoESdHpFOXocEzqgsiupANKSGxrphzEcoAJDQsJabCgLCChqdvrRyFknuJMZGqmKiCYJPkWOwvniDtiPJNulqSDkHvVqxjLBbzDsNahgBKcARuejdFDHIRFrjhyHxRelUkinkulHXPatkkCFZrwDkHVkAAjIuXKFeJOTartbNCrcdoIXXaIhfMzVlpHbxmmZpJJLyBlJGbxvDORxpjURdRrqcUpMOMGYonAXUDqFScMDOyunJiDlZVQpfzPmQsrwglPcscbUSjGZPQzKVGTcygQJbJSrrPrLrLNkEdNQWmCTBYZQcngvvyjmcCcsVXNiHRvTjcwiMQKKLEWEYDnWLKJSjaPmjOWpKOwKuFZenpqwwdWSOsbMTobDbeLAwDanEHcChWvYlQdFzMTuzqZQYjqxYJdglyKxIeVgrDFZigDndBpbEKeqrYTdvodNWUfwDfswJLKvYwjGzxtNpYhGvwjaBgzNETmDmCHBydyWiHCvaXRLNNFjCsiwRUWAXmpXyyWhIHWqRpJGxSTlxTfINBTEFKsbzwcOwroaVqUTpjHbrGLQrAnNUdeahkcaZHxCrIaVwCxYXdzARyMdXCrNRAZfLEXGrtUXTLVGchlgCBNPtvLXcCaXpWoaOfyHltoYzXBgBCYBeWzLkGLsNfbWmYXVFnrJfItEaRRlrkKeXnEJwfgUaIJrHtgNAyqmGUwFhCXcXBrgcoXtljlAjnIbdYPXbPoeiWehmYInezxQbqLXJdrChclTBYpPALHJNLxNvXtVDofqQcPGQfANctqAFNvAqyubsBookReqquadAAXEueULiRNcNVPkhQNzrWhluScOINdAHdWqEcKoIvjbcoEfqsKgNzSlHmBvCFgiRwoZleVtnjqtavkKbEKrseQkQbNzECqTcGaSFpscntpEIzdImAucbzkUvswXRSSvknfailoMrubvDAOaPYgMZHBiXSKBZTmQJuZIlUKxBHBzkigtpuDEXkVliZiuVboWhbhtJEHtDQtAdmuGYAJpxRTrLLlSndfMSGqBnMhCekZXRzQxciLxwGRnFMGZEvbvDyKSTqJGopBQjpEbyhXFhShknqXiEiYFIzBJEvmXJwixxPYYKtVVJWfnPpYZVorXBUtHTSJEiOfWhtrpXZlvEzHsGZYXMSByfYmPjGxoQODgZTnGluombJVmuwXDEUZZLeeRXrwhUXEIRsrISvoQBQFZXmaMRnKlmKkKiIZTJcHwQzmZCmbEuOMhmpzULytRpTGYpgpZMvvqgQbkKfhAXWHlkWwIrBAKyEIvViueWLybcbAxraITvBqtJFpnCvkOhsdXMKPejwYwclzBpIvKSJvIlKrgULaCtSNrdomeZjpELDqiRxbbKrWwjpeTWpuqwYWtBVurNIalYbdeQybrCQyFoglVzJewNmJzkNKarHBKrZaSCmJXAzTGjyoGsuXASqyAWthuMZeUVmBugYKsvfljOoBGRWMsIgfRwUzgHHvpYcuXuMZKWhfNpBNJTokvSjdeOBgZfHkRuwyirqrUkHjsSbsgdUYfyfalEBAsMUSZThbtYCWtVvibpKGEqLoGyLwzALDsrZoPprxKVzMfEsevkNBITBMTedcHbzLuwLiZJAvtsrxRuptqQjWDwQKJlsHoropaLZExflKtJhIjxKmLRAagnqVCKsLbUyXHiBgCdkylKnWbyFbmodDmCRWZVQyjwWPomDrHyFPwxJPqYrTEaQqinzmDdNhTSjkuxWhJKUoctnrVHppntorhlHRFYnCITfHJIchzvaJBqmkzqqccaGtCjqJbOBDcsOkxsXsuedBuoIUfZBSTUgbSkRPIZPHAMEkSjuyskSUTWKySnWLjvQHJHGYQVlsDGVvjzXpbLClKvdvcAMdsjuagHeJgTGmdNXThWhyKmQaDFCzEviHBeMOKZxWbriLsKmEWiOtBTlWGhwShBiMdWyqpOBaSFlrAhsQlIwDbBcsBezUBJdrBmdRWCygRaSOwflnuwWhvIDruYDMEtzAYMCVxlRWQsYEEhZYdokNOLydYhlZJcBSwsSnHdMWINBPuLPHZJxzqEmQmFKjJFgVeCsTXYQAqBwNMrYTjYdkdBLmRYDdQbvjXOlUTDkTHHOCdBqkZSzrYfdtokJbcNSTtoddddfuoanSroXbyJFjNtCNLNPKuPuRtRWWtHjJrHlwKPCBTVtCOuGaMVJiXdGinuWsDANTkGoABxFCPIfIXmralNzNtaFbAZemByYdYrAiYvnRkzTcQIiwADmSAtergZDUnlvmOwSwhKvuhApICOzfxRGyezhQdEyVkcBHxaxVRPAFiKubvfvStcOqKeICVzrJxmvRygdywpkWTniybrMNrwaxDTssjJmwwMgEpadiVYlxPrXrltkeXjpmvThsAHqGzvFiyeIdKEtDFUoxxuXUXhxlXuXevtYHoiIZuuZpzfPgSLEYweiRnASZVoQfNcgSOLuNxjRXHwwmSVNlOkQgBQGISASJjCPKZUqGiZpwYHTYpOsrQYcJwtaQDSVzkySLfijXUnVoAutfjiQKjSYfuDskZyarpvPAlfDJDWlfHKztegTtqvccKdRLlwWyPDcfoUsgGdWaVNecYMcwNyvzbYwnKxASKLKRcksvixFXeoPUUXHSVTkhTJRwUISGGkFQVDmJlmOGzXwXYQKnjKelWhHNORgfnrgsupYujGLKQLDfkuAKTYtOdqCUYnGNaZHuldutHTWkoDnLkPFRbnBqwpiZGSRESUFSAVayyGQXoZukecEtGgOOxnbrkMitFsRXrXkgVmhQWHlqIaXNCOSGoevikHZnEFHilkMSvnFsAeTgADkqvpWTKIwgxdsjSBAGQmvmDuaTZEDjyjLxrAgKEzTPpoPSgZDBkPPySDemBxPEnggzebpJLLxUJjgCVWUxXzPNxYebfKUVdBjIXDjHLxTlJSrlarDDrWqLSLqtDSHpFYdWcQiXgqwfCkGgAenvSazXMmdmSDiqPslSaqcnyWHyiIJdsLfRRBabuIpMcKJANPHuwPcVKjVSMmDvoRAMbiTQGMRuBTOiQvorJrUXWBaxcgQkRhffRCMIPeYAKjqShleiooYqaekUWuXlSrdcxfcSiNRKuXZOwfAZUbPPbEWEZpWfOBPzZgfMehprsdtIynKjkfCHLXvgDqHaDJTGwxwwvaLjVyVWnEQkFiQPLhvYdYZWyPUatLOyAwIDkssWArHsoiHxYTjhjfUpbqoVaaavKqKELFrruODcwETOwaTmwkUlFTwbrYKjoRMYIUrHNTsZPDJxrQlHQKOxxKHABqVxWExPMrXJjSTFqDcwKpDLqWTZQtGScEQAOZMEAVZZLANZuzZGWoeHXJFDFdPIGLIvexpaXZtUFZbCpZuizpVnPThtSTJHoSlfpvngvPqVGDevlQyODzzLxWQYChoRgdCoyHLiPazAWYOJBMVZKJILlNZhwKCjePoQGDCwXxZUGLDihkSbRYNHxRLLsxrreFDbaMSqXxbXCzmoAJlEozayLnOZkKskffurpPfitvGJbwlEtSeXxpuHJVJRVfyPuRkJxRTGhcMhiUSWjvTHODSmKrldjVrEkRFXvkDEprYyYPkLgPXrWpuRKRHwJKLGqYYWWGIGdQRrwechQmssQNlfqDbmUlBvEkGJRDzDvbbyIPoWtVovWkapaMqskvkJgvTyerqbuIYbUsMjkojAToLDimoeXLrmxxqLRCdWmjXYufPnDLoCWWWEfdjQnySoAxeRXIyolmMnkxDNASlMoMEYrSnOFNcMmflVNtYmuPXNkbOFktzvBOcsLTIhMeGobpTMUixkQkkcCleYnNhCLYGmvyoomCFbZrGmVfwqOdWYXXoFiWBRvtiOdrVDLkxogBanDUDjcdIIujtyCTwINqmpDPJhVuTHYwGJgBASPGtcSngvsMXGQZJKyucjBgouHhbLCAsbVtDgjOzJjSQeKaTXMjOzxHDuQFrFwjxEBPiXiekXqsZgbPupZSIFtYtAETdXgkKBHQdipLDWgbQhoeXEfrQyATeIamKIQkFoopLtilxwZhthowAwZNujVdWQdHuZPAbdhSzCZWvHTqkPoLHQlMClhfTeiKkGdyTeTcwCQVubiuDHzbRNOPtBzzZNHSmzSRBViyMjelHtMvIaFEJIvrSaZkoaYKvQvvSUxMlxKEXIiWeHiPtsmxsrHwUVTQavmLlGcwALyAAkvZTUgoIhfuhKnVBawHZuURctnYAstSAKBSiXjUigLJDwBMTCxNBGqTZTddRWvUlFZjEHQKZzKzzdgXSgPZkFuSpfgonUuYSvaCizxkmzNoExRassdLcAvDHWFdmHrOQHOJukusLUvRZersbwfpmwktGdQvVLIrjCnsrJtkhYJDKpfPktgkWphWczDFynARYdGBZdFGLZvVRdVVobhdsNXgGOQfLfMgGkcIEgovawRVlnPmfmtVbPwRXCBkpZuAMTATJHVndpziqmJlVYDiQmyxmKTGTMjKBEYtHJOCMxWxexufxMcokTriMnaYxyqzEKSNYVIpcymZjItSdmVcXlgBNNpzeSkbdckRjtDsMyAvBjgrcQSpLrGBhjcNBzjwLoyVycplarTCeUbhYVPbvaIkMZugIhorkkvacDbEwMqfYNmvWFOuCIHwRgyPlfRwxGDBYXbwQXrJqUqRaODSdZwSpXxTCgGirpoNsxMMDVXqkGnkDgonJTxpgvyZQxMRDSuUXVndvEGPRrIPWgYQXwtpFwnPZwZuOphVXjcUfvWIZGdlYzcofnUwsTVeLKdtrSjYql</t>
   </si>
   <si>
     <t>2026-09-03</t>
   </si>
   <si>
-    <t>23:25:33</t>
-  </si>
-  <si>
-    <t>2026-09-03 23:25:37</t>
+    <t>23:42:26</t>
+  </si>
+  <si>
+    <t>2026-09-03 23:42:30</t>
   </si>
   <si>
     <t>{"key":"value4"}</t>
@@ -506,52 +494,49 @@
     <t>&lt;root&gt;&lt;key&gt;value4&lt;/key&gt;&lt;/root&gt;</t>
   </si>
   <si>
-    <t>9223372036854775802</t>
-  </si>
-  <si>
-    <t>tm</t>
-  </si>
-  <si>
-    <t>rJ</t>
-  </si>
-  <si>
-    <t>Pe</t>
-  </si>
-  <si>
-    <t>Gq</t>
-  </si>
-  <si>
-    <t>nZONAYwBQzKIzHsslvIJRXWsbFURHqVzsHdwz</t>
-  </si>
-  <si>
-    <t>WolIeQfIccnquoNHACEhWpdJFhVJAzOznKegOURTjCxWxUeqHgukAtesRIrqeExkQaNPZBmpOEgwXVErXMQhlImqIMoGWBCKrLmX</t>
-  </si>
-  <si>
-    <t>OCvOyjNXbyAYnixOlKXZjOACqXJvTpkxzLEyQAzodmvcfuRVdxjmwTXQmTmoetNYcCZCiCqInAUIDxgzwIycKeMIdEuyDnYQEmXXxQYNghDmJYdXgYHgPUumkjtZpZtQpHUVhNWqbwRWhEfechO</t>
-  </si>
-  <si>
-    <t>wukMAbwNdrfetgMTZbITFxYWZhfaCnPriuBObrfdNXAJlvwkUhiNwgNgLkTLBIAvGCoTnYvcelgRlrajEWQlwMEiFIwwSeeIJDiaRPKMspnmyKUkeGHHHJSNAsXrNqogAbLcRCLLLRhABYbIFExSiVrqRyZrSejkqqZUmsjKbnoswcjjziPrBxydCjsQywBsVqHysOWqubJd</t>
-  </si>
-  <si>
-    <t>pUTbKpEYhyPjGwoFnvVuTfCYxdyRyvqZeOBquxSWhJqJdvoRDHPYWUBGEMvCiyHIyHKJDEAofzDQZVzobSVuZpWxYKwlSijfbzivwzpOrfDkfAcKmivXgRxHwWOXPePoJfoPAJxAJTCEKcHeDXDPbFVQQMTFCESNWovokbHbodJtDGOLJSegaBpDtKPSCbOEYtQgMFesYHTBdCpNhbNaxvYmEUvWvsayLXZgAgcCIijFsrNnOiyuluNjeIcKSaEmWzknGQOBqbGUOpAqDAwabKDkiQMDEJJYVkJiSdMlKRCaXyChUfBipLbqwjZeNSnMCtwgdxkSsAzIoVhDJmhayDMWZxbSPJcansmXUhscWLmXLangDiMcvdPTrYRQwIqxAOSJGVveDGoTLsEFhrRpIFLIwzWcsHBBwBrfVSuvPKYdndEQnyEKcVjjOUdKieNxXIOoZDuactqqFiIKicuRJmPjidHozzEpTDQQarGyyNiFaLVPOiSZcaTqzvbRcEPNEfCMYurWNIZvJCDwYqiNpXWsVsRCEEaaVpTBtwQiXcJynPlLBkEXFIrWzFvnnPPbJTbTCfatMunfVnimvyLeTBkSZErcQxxGtUYZXJgaMiorzGbIBWLUAcaUnhzxPflUolyQQxoaGmDJteFGDwxmBazPIhcwPhpNLwlSLXPlniiHZUdNjsFrOxrGjfwdHkBlZqJuKyMrUMGwwggIJLzOBXDtQsVFzgJKqBZBhPrhWwdqInNKRqmAQEJYtTeVMnmiIGyBUInnErSTfMBrcwKTAvzNmBGXPtmmuRRXHiBbBAqmlvWjIUwAFJhHLCJtXasoOQoxvmdxOFjrfJKxKBSdFTWckWvonvRZAhbmHCjRiCCdAMktpSKcBtJtQlWgPTZTFsrbMRxWrRuCOlFDjxAxLivJxIDtHYZqJNGGEXmpcoEzTbWLAyiopaPGHxTHjKacoQCekgQHjOYzVBxUJelBrgXSRrpnaAifOwnGLApCBtOacZiVQjWnEWVWgasAdpXjNHKWsRhiKbzLDpQHGUVMOYOxLKKCgHtqnZNNdCSvYOsujfsVYOeVJGmDkuRaNOpeiMSkkVRoOrbxmlKUCEZgpHpFVkrFyuIxZIJyXrXPSgFFddGQlTsyMhApDTBfgcRsJzfaSvOkPDGTaPLHEVcGfmeyZvbebPORJMCTIAcuoCIjdlWLbMdNmXmNhSXdkeasPFcIURUuiDlPHugKHZAGNmZtktdMjmMpSZvVYTGkWUtmvcQWwZjOhfXmdEIWUjVOLzKJyJnKoRrnrglTGasTETylIhMcqladTcTzjGnMxxidvlwOwumQCmYwfeCLitWKegTuUUZiDJGNGKThXXvrOzOvBdECIVfXMgrtpZspcAJmPAlGLNKMBodgqQYCLAWWuyzjcrnUDBVvJSorNMCRyZFkVmnibvNhiAlOVtgipYGeoJHlzusUzcYLVPnwzmtWhkZKjqFFgFjrQUqygsrBaWWbsEgMXuuwCFraCBkzVneNTSCkTmiuFohvupopVQjTEygTAZfKkTWShsuEWilPEGIwkiAcIOAmQnfoJetdLYnMjfvBlalxoLbWUVzFBSlwgvuCEGLmgmxZQgZStJqboVdQwoMCIifasrmiYCLfeoDsRUYMTPdcugMcMXWUdMKRbahtDDNtzOJcPbJgNvHVafQbvNqwbbuVdMgyKGCbXurVCIVofSFkAzQnPjQBNqBKaLxJzLkfvwPMJIZozgFVSJHfMJHIoVdTXYhydgoUZSkEGDCllcNIdLXRCImZwJoNAcdNucPYGmZeIPVReXkmtxVQSMuiGUnlSDTGRKoztPAlvvQMTCXisuLrxllzOPqRUIgZoXvXUCxndixJIdryLnfDImZPsaFnbZpYDlAZtJtWUePysktixAfMyRKZikSGXSOwdEEprrmkAWfxanHyHxdmugWAIJDtsNfSkbctKBSUeetXDXXwMsRoZTGCdELZtJTMvqjbUCGsHpruTfxJqsPWxZQjebIUYevARZkWejpGLMrVYkjKrDBOrYfguglSFechXlpSFrhjLwkGGDKhDbuhxkvpxcTnBqFImzJCEOibzNvHlhRPfDKyZVCFuUujvqpnVYPERGaIeSkkrTRWudAgeWHbwKlFzTHMLqADOTqYwqaYgWTDUKLmOBUnGgDweoinVfJxnomCDElZpmHDEZLSCClXArnUKINsOZZaWGuIPnztOflBWGxVGvwZDPFugMHcohayLNeTsBkjbuYjlqclyChLOoCcBmdfRJRPcTYHbWIrAMHModrbOPdUnPzGwlXlFOierUBTkbUVkcKPUVlulsirhnvNoAcboTjSTTbTCrGCrXlfPJdUazYQHakxnyotnTwNqrdqYDndaNQkHiaNSqHBVLxOIgmGtzkvCLeosRJqsruCpRvDpQbBZOTaiIvtbWYIJuGttfjcUUGxdlALAPAIQRhpcyYgElJkSAaGhNefJwrRebrBhoYGnhWMbOSjXmPIDAONAIgcNkqntiUyKWjEuUsmTqNzPbPGbyCYKeSWHujkYNmDmhjGUQwCaxobaAsOOmWOPYYEKqVsKbYrRRJJDYEtMcVRsijoZIEsxRMFkAIWlRfNliJTmuhKKGoJdkkjJFHhSJWSbquOkTZFxDMfxhfMqCdCjAwLjWdokfBxOoJRQHBNLYkYyHwdvRDgRnOClZFRLVFSNotZBuuReijyOjybyFQxlPnGStHLKWXpIVsCbSjBBRNawOHeSSblYNGgELyfnwpHjHBhDUGAEVGkiSbWGCyuGZzvnqPIhWdcnuEemfBorRHUnGIDWhOCiVapAbwnnyAeBKLbOtLzPkdvhbdwqNnlKSvpdaNtCsHlbwDUTQjGQnSoFsFgAfUNJwpwPOprZnrfxQeEpfOtcLdLOgYSSSnLttymCPIYrFyzgMqKiYYHSpjXallqtrqEWDQUKSnIDXuypNmvnrhpimCMudWloCDPkdOQEVtLpuhZqdzHvhcVRKejmmFkDopNguOvrfVrlqJQCbXVrsSFFGkrSYERAPLHfWUNlngJpqvcjDGsUMtjMpkiJoKdhJhdWcGoBJXExtmrtvhdBXVmhfOhiYcCbBFoVTqrBrFouEaScZpsuQAromIBgrwdIGtuQZkbphFUqKvRaKZusdVYyNIAqCAfjwVkxLuhikAtovzjMUTVNbugVnDppnoxBvaXuqIvVqCGnztPNSaMYdsxweviavCXiXnhbuWzuhKyNooVEDYTbxOIFpGVdoqKSJsFMjpOYNrMtEvDoeIKhfGQUDRRtDtXQnOBrIAfBWIxLvBUQTYjgMlIdsoGooerxkXNVoUsVHPSpDLcGTEOPDAMmFGLFNSrbCwAocpzjtXZSYbBBtkudIacSkvbcnOEXhNdWKkPDkLgqUpbUlEdRxLwpvOSbcqBUoOPDhiTCJzwxdqVDgNaOYFYTTrKpvqhuVVJExLPCpTsVKTAGKuGySamVZeNFNJCZZoEAnDLjrHJxNIwvMtldBsZBoTGpIgAwTldVFNsCMPzojpyfLnHnzGTpBuFCccKIYpjWwiBclcozBCilCBMeATMmdyRzJrpFJyeAjUTxvsMkYkMKiWrlvpYKJrdSxjcrlXoHmtCUiltqMsrbDGjBSzxdMyrvjZcqbARPJeFnNBDRlSfhXfSCPfQHRtGlqfzNBgtOeeWuQAJlIdqhxhrnWtgAjbkgtySfvqyQyzEKRPdiwjeWLCTGlZVCbjXGsiweiOqRfuhwIszeTYOQLTlTJTohmZWTmvGVaHgDFQfwwxrvLLDXjQheIqMGxbtngVGaNVJgfOZgFqtQsCyegmcBxkRTNAhWKYsQlAHpsuvjIUfhhdZxIvPYOwjAcivWdnTICDXfmNrauRLTxlslaKIxBpMZOySEYsOIdcisvWMlMdWwkoRgYieLVixWOAqQLvBeruRDjEGrJXZKPYTPWSYEYLOUhBbNoVDDbiRreLRIIfrTxBxrHIigRyxQOsCandEHIYnfjVHvIRNtUpPWnGhWadvOpBiSnnXXbFtlHORgCwqYAGcSbmxVAdQarIXncVigxsxzssXKAogPNvxIVZjxOAMyasWNHYLaLJgLcrfjzBzjYXfiyKnSJVFFixJqLShBoJtLxdFqxByTpNHfyEPeYUHKjjhRIqcOyffOXrubwhZVUTvGuMvWhiWpUvBbixRtqvBVtulplfQgVbdPNVadYClohZbmVxPLkdfAncFvKTnpqbquQHjTUmNwGHJDndJZAWdjObfUvmhPbgthjvXVaqBjyRPmvjOYNKdpKzpkCgwTwlBxVJxhOCzkFgosWptnNMiBrRVexMaCYqPikqqOozwCtypKoYuHBkbQKoRWWPvtDdmRcHtHZyVlZQWNCedAbhoyLnOUYTXMaWjpUyfEaCCNtISGafzDqJeGJpfeHrjAZeBIaQeRZKwsIpDdUpKnqtmzhhIJxTeLmkmxIrTnjZDsIqzGRBjHRMVWebnlWRUywbyXGHKOhpjBWmBDERNkcYfJpJRFkuEAVZmrnhNsOwARKRWZMVhnrxCbEvUlQFaUPOqOFFIeaScqRetZyNDCFpzWhzfBPzgWyhmDcilrfqNSrrozbrtCEwIlSkhhXljsvxmVCfXWutDmhfpLOJiwnqLwoAQaQyyssKDRTheAYVLOluVrVTuSDWZDuESNjRzotMQtXCTikGLwMwBchHWHedMpPtfrQmKQtQqdtdbSLZmIpmgnkZxTErqDMNMBIIeoLVnuHBnIMdFjZUutjfhyuQhJjqEAvGigIKpZZFuAXxyNKoIIIMtZLMIsUpjkivvceBOwfsXunEZuBavsTXbNZPqrTMwKNefsXloaTTfKbiyzapuIXNQxWOdzNPeRbitTOgGUPYfWoLjWkkPFZzVmxTzchsAPHCsAlUOtZovOwyyjnswFYdqKheHVrOGynHuARuzNqbKWCQlGBapYJxfHXtiAImgskHsVdvGcqnCVKdkYwqZsbKTpBLENBvyvDXujFvVNtntvUKogozCRRlrsoqOXmUgPFwNnZSudpbTNxwmYHZGeTeAfmyByLfeYBeFsghSkrtGSBiCZDPUCEkQgdGyOKXZmyFCejfanyLrytVnRpOYVklwFEEnClOSRODkVOwSwLDNzIcrKFeeNbyheqMIkNrcTWsGdkASHptANBGGlBMbDAoHtJxsPhTVonxxnKCYYmzALRRSrNUjwwFwpWhNVihWJaiiwqWEwuHNbtkTNzgPjqWLTOEFYPYyUCGuppMAIRIYWYCBubkNHVrxtCggdZuppToolGewmbLsBJELxQPDeNvHRiHovGNEVuRAxupqtJbtcLfYBPLdmhwpvBmKuYzduJuUmXuovpdzQanuXTaCNZAwbjBeHAhoCXxVmJMFdsftfEJRpdmWmqqdJFAMdglqBrggPUkDEMFPMmUpimwlxNTAxJEeRyrSOHIEnzxRtNuUCDDctqzAUWwspiVYfJYEoQPxiBCgfpqAYNWnfajmSIghaNQQokDRAVRzdsdqSwFSNEQkdRwhaQaLcHHqhoFYDgaHqoPTaAmAoACiaENiHyggOJybrOYwRLmrCWBTcJEhvwFlWqhPdPWAnirHVkovGFycNDUbcKgNYBlWHaZWIyXaQXWpBWXnLaAfuPDMEvfHjboFUsMmisOkNSMmNSgjlhjZtVdjAaqmnXrAFnSkRuipNKosYfLnlxgXKfPKrIOyAkKvrXdRJeksUmVeJrgYiBontWjXWAxDkzyANYDOiKYDiSNVuCTIyZkbgLLjPmuZFzTxuxRZBHxkYJNfZsqCKZQIYBOfjpIoSpkHaHwzaynoXrvKoDwiMCZSpIuQrJMxdVvFeWPzSagHvQqXqrlWaGqyWkBUaICxuHfpBlhCcIFDLYurlcXWlmDZKOkmaKfNTGdRuhWggGijSsSysGUxBPOtYSZDPfjXVXEkqaznLBEHEhLBNkEmVIIecULJsuQcCJBpnxpCFYEJZXVHdTsffHtwSGqMVQCcXIlvikXBKDaJdAllkjeNQaSEzIEWtoMRNonGAhfoPuAyBqNkSvmenEqDiSMfuqiPHzxnFjApZVRTIqjWnPxnNcoLJKVTIzqTAhqtsKwuSEhLYGCcVXyJZefvRyTGpdFHDsjnZupFIJtMLYXeAiFbYYQOwvGGUyGYkRURMiiapooSEFJjmowPaNYFQFgzaRrPuSnXCZVrztUJWNNGsacMWeAcTLNUJdzbxXqVXtYsOiehhMwSmfDnOWmpjzwuAASUpEEzfazsZrKroLntSSDqqnYyRVsavoipUZESAQuASxmQJCsHLsKQmwKHQmJafUjhsULQZRpxImlAqHteCWJCZwxbliotDCKxOvKUOzNWGOcKKqJxzHIxVMwgUcDgnbccDWPEZjOIVFDtkrqQxxKGwGMzdpSvGcjNZLtmjGcDofqqMnlJaiXznUAaUImhlePNectcrVImZqGIbeewIqVHCHGMuJhjpFJZBRgKTsjfxaGnhXZOnkRSUNDoLlXcdVgqXSlqMsjmCIVEJtxqoPoLvgmPtLKKWpNTJPFKDxcrrgYIFQQDnwkveTODQUzwsYdNJYnARbhaKTUhYMykBRvwrsmiljwfsFjAFvUZZTAUswYtuPpsHdYNkfARTasxkrFjkxpTEIgAJCAcTKQPJOPThsMijVMCUJOPhkpVSFhpPZekCKWhzJOQcLyJysuASxZSGftCizjjNKQyLXlRgpIevAtyNFCgqppmLSiTtaEpuihJahvCvWPiiFwVtcsatjluRJUzVUQVqcjmYUGhkwHhvLRgcBaxoQMNWOhJCXEbDSpxONsjAWExIbeYnqmsKfjzEVrlfwDkzwHtqbgIsTiKYxlmCYTkoSXYIZRzULEXzSDhqRvIITMkFQlseVfYGKhmCFwIkopXcxiyHOIOiHwhjCUDkuYgjjxoZYdRSwztoZavTqwlgQeqcjiVBRIkJULCfKuQUNqBPBCJdcFdkJaupTWKwKDGsLyNgcoLtjcBBXlUpLXraUZPZtlStUtfMJmApmJnlkUcTfSIJUzgoAlbLKhcOzfqCQmRyUHqozOsXYGRXSyXyNNnVMederTYYVuODcJycOBAXqEHZFEnNUMuENJJivYelAdmQOxYfHMYIPacDuDMaoYVDcTDPiavkWRyBjdsxEkcBRoEjoeIdTpxbldIZbRiDDyCDaFqEtyGcBDdTjfKikCkgVPpiGBfuMgUbsShvZieUWgLHkNnThfpJzSTfobVdrXjnEyqQBJhZaMMpMXWTNEMRYkJxAbwHoLQVNYOrKvQbdETTmagJcWZRKopmNHyJIXbnMCkcYQhGAhZLTmvNdkoyfgjSPeQjsDjfCSFyxsXfRiJjaUHMPiSHVFaEPuLoLIYWdGxUAQCuSrOVUGRzXzLmdDnikMjxkowwKHxgwpnVsSEIGvErGrckRBqYYUuzRGeSMjMXkTJyLKcifPCQMcSwUYIigtlvaoUaVFgVLfQZDUjLqKkHtUXQYzMnzOUELcPLXUwiIhscfNyCYgepuevSHrLBpEJsaFYuycnfwbimfroLStKOlvWMraHlrRMGrIbVskuFEDoCHaeTihecrebwEvxmQITPkIYqmvGmDJJlHjiocujUBCeEhWBsPdQwjNbgbYCotpemCPHGIcoSDBLvnmhXlHjGCjiJXUUENDoOeYbyRqmnxpSfZLHlaEDUkZElhVTQdASmBaWlqmoJvMZTUVdQiSyXLlwdNhHxsQMRUoLFfGtqwsOIsnYsXvWbdamMutQUQQUPbGapdksABkVOdWShBmYrCnyxZiTDwqFIJqZVHjZPdOMzYvPrmSkAWkvufIRvndncmkZHACwpDctvKHzMyDDANZYHVevsDTFjAndcNJbiSnAAxcqlCGyjyTmZeliZvFhBGwykMuCqkggNoAMNTSsbqmBRmfuOxivaDJTYwsJGEUyLrIBiphsdNVtRTZzvqlYSQVwMUgJRSuokDzBYsgTFQSSpGVfJavfeVRNMkZEAQCEgZASUcJRVWKqNJVbgCQwxQTzblzJFoxNFXkgCWfPTrlgXVHOtKHBUmizceaTDfpwXsJVdOjlcZBRAdiPMBpXcxlmhaVUdkAMxtJsmzCNcaSePmZynyCywhMHCQaDiaFSIixpaTuzyklQHXJoroeHgbrOADvOJVPAUXshsmnEBWHgyCcqEgqGdsMzUUOGYrdTMPkRxGXkwEOHlSmviDTQrPBrNhItioUiYwQxsESqtScoWYDTQRhuuPtzZGHIlOHxgDWFJRjhpwsncfbbVTVExmEGHalaqvbsUBHRHwRWisvJVFubwFRuEtGJuQisIhsMayovgJhNLEdccZsTAwSeEHGPReBuxVYgiREslrxqdogxgfMNImqEyXQPSSDWShuyzzNFDgoYMUJDFcetFEmEGdHwpxZgbOekxlxhxqhEAmWfeIRgmwccvgsaXupyfRCqPyLrhCuMAFlUycrmJPCjHUSoiAhSzROmOlapPAVlVnXSOTZilRmxXUZSQPMsEDJmjlGIPBNdWevcRgQNrDFZLpjyhfpMdRctZZBrFYNYaByvdDFgrVeTMqCOgKZdwPUxbdjmCtKwgANNVxYOADhPBHakxbwkaAlzwcjBHcAnlNrbzlYpeOdbnLOquwmdyxLCwwwAONNEpNZfxBopgOsBfENXCvNRbcRTZMqspdFBFUNBRjmMhiPHJzYoRsjdHUFDfNozKFMAwaLcvbxBWFJMXBDClLftZVNUttgAzdIOoxFsKPThJiMbqVpMcphzHKgpkvsUSwkttwWgtyxZPkcWpcvjoBxLxpnUgEZeZdyAuMgdApdRBPeKCYdulDVxXutXsrrgLpKSBxAvQDjJJLuTPmNNPovGfdVmfndOzmHBAevcsUgUYwRAkArcrMgIcVvQogmmZDGcNgzDDMajgxwlbxuzDGGdOjELDYbybhfURXauZxGthYCwIUxhBRXSETwmaaZqbptKuhqiwQtRlqMOnWoArAJtsGMnULxQquCvEijkjamMJmUnEtuQftnLSSYiCxoGXnjtZIEURZXVunogRmcwyilvKLpzlQOnecOtzNWxZsRcQRRxGVPWIpNBPtXsZoLYkznjLyOqkXDJaeaipzJEAXGZMsbhJaWeYWZinIfxBVzXQlQYtLrunxzetmTRlUiZhxqKVWavHQDyxpjgmoraSlLxNENBsRSumiDrglJAAwWzVesKgPUfIwCWQPridneslQcIzYucQwjgUXpBMrrxlulvNCWehBhishKZGvLkyMVpLwrXPUevCmoowcGaTQTALBMSLLJsmdWNcvopLyuucoNXdArPzCdtxWnVUjrgRQghTjPUeFelxgZNurHaFeVCrqyWaJYwDgZoNgMvTRqfmVosFDDtiHZhoVqfRaoffjBgMDVGbAeeuWrpGrcltGmrWQwFLgNqXVjBpzGKESsooxlNCDITGVbRIolnKKRFrvlFCzmwQcXPqTvNGoQQVyhxmHBNwHYtznRmIVtOKuytJNwDJkPDQkXenyAcSXqptAsbImcCRaMjdDWrGifGaJxHavnaACAJIAwMRxkfbbcJcnuObKbPVDrgZjjXoLncHDrchJdLZcewGGXYZmWmwVIbiPSRxOjhLBeaoqKUgBjXfongLbtzZQhiDDhcojQlxNfAaiWEGXWwxBuRnjQRbJfZhfyRNqrZoNVYtDiJREJDjCVXvjQOjSkDnQuaagOaHxcdvSWognupeuTaVgvcRzlyZGcwSaKgRciXDkLnhMoYwXKTbNAuggdvahZfaCTdPYyAFrWPCvUjPfeAaePPeEVNppdBpKQYtTUmSraQPosJVNxalweLlvGzHUnECwzHSSEWTTVaatHfXvZiHgkhHbUQPghYBBnYbZiBbuTXRxYbWqyyNofXAiprZndPeIdWnpwiYPnloreomYfiioBwKUBvwnXOjVhPbqLcOSqFVlFxiWAEyvuUywXDDWzQDAxZfAXgLLNyIsDewWXMGokAjfetFuDfcjQGtgjdAMKKeiUaAuEvEayOIfRbuGOQZFdDOTXuSFKvEQQfjTKnnNIuiVOMIiLgNoimUbThkDUDpVWaHmjewPVrtUCLXsjmffIjBmIPaSgMCrUlHMsUPkyFOiqHSSrbpJQOCDiSUeCAvosZXJkJAEhwztnPnStsVIikkVUOWZnZDRQYZaZvzfNILNxBypHGZFuRSOEffXpBFgzOcEtmpISOuqTkEuofsQfIwhwMKGOiecUEYJxTakwMWVjXlsfKnfnNiaVXBSkMXWltscnnmiifbQeuNaXqzKeZsYrODfflDHnXsvGhnezwdixcBzurqxfuDhFtRTSzaQeOyAZoNkxVyCgUhzVVJwiWPWvdzrhmpiovWfzIAcOYWRbCJQvVlxLQNzjmCPCckNSUouliOHnvxtiCCmvtMNHWCfJPBmLwaRedpndsjnIsSHKpGMQiIAINthsBVreTfLcikSlgdkSpPyiMqmwfaACKHGRZsemBmqItKRNCLLgWpDFYZTtiavFBZTKkOZRhYvjwvNbVcbIbpojMtKDUUKYEpwYlokCTLRkEWypJaywsfeyxoapeLSgSyzjodpclPOOOWihIeYCbGuJMCMxnHaSAGEdTogjBAjlEsRlqTQIuUADsDHpiTfPWJcnYjtPfwjtFRXpowqLrNIVFmfwUfeNEZhbwiYizVLTWKQnAsXrPWwgppLSfcKUDokoXvTrdnJawwxHnegpPfYRCFbUNKFyutIOBqVSporzIdlLduhWFhsUnNtQXvjLTLEjDLdhWsvKOhJPJbMIOLAKHZLrHJiDyZWGAMaOYHbsVrxTIFkEAgrPiNCnaRZrUFyQoXyLguyvblCJgDEgONZhgQjbBsbWRDNvDiHbrqSpPpEUHTcpqWCJprmPiDqkrrFbQCzBcFlfsepihNtjIJEbPiQQnSMCAGdzAzzSljalrTDbQUKWDqPkCDchMMcjDZitIPGMdbHSgizuDtpbPeHQLwvQCQHCVGLJzzAGzPHxkTabhFeIlNAsNEfbaihclFqqwQHybqufQxaBIVQHlHylcBXMDJXtBUdBFCRIAHhaiemhDpmVLcUUxbGOUQgIbtijShbooLeAAEWYBlmtjNTbgHBJuxCxOWbMMJppeKyPSHldoLqlAnTHWHGIVEDiShxblMpxPpzgWbgAAkYMglXeeYTTsznorHcrSAeqeGDNBEBcdJHbKreiTrcRHtkqVkdBvIzTnDhKsfzKBhjfwTMxACIQvYXkPnwlZbSfhNWRetUeOelidRlsEJdwzACCkUKxhHvHcULJlFMAkGdteJHhyKFtPDfbytOgGdLZpPHxSrgaiHnXlXeUhxZVrBJsJOFHtDIANPFKIAWyiULhQlnaUMEoRFTqFAkZalpMAbaPGPztvViAUqtwrBdHHKjXPjmmvaQuUHcTIkPIIdNsUpeUaSICcwjuElmueySXPGolmLZUaTAfGbSXcEyXanBtSmQoFvNwKiwzQIBGpXoHxYNflyQOxgLTpvxXOBlvoVswSETLtNUOFLMhJsssnqciMmgAlepYlLecopXwDEFtEQIUSkXfDDWkHovoiMIuAQqCiweSPDAupAKYmeAFTyjOBziRKxDQJESELejcnxEmoImWHYnbmUSVhFnkQsYvcUxotTudwRpPOQXktdcikRWyNuHOBcEiJxTPsdAPKdEMLJKsyccEeDpvgktYYOEDeZyekVOAmmXHqxGdcyoBkaEBgNdSfYTqekzwMFeBEQtOhvoymRtHqNMTEAwrENjUdQaeTCewFlGqlyiaJVzGlXoYsgpDxzCqYKoLISoHZcUgWuILbGFHguwLXTsbXfrCnOdiKLkMnKtHHvJfOCKOeowLJIOujvxqYyeeAjzBXbDXhtdIwOdNlCznCimSiTcnliKwSWBSCsFtGyFqEWOHwiFeazvtAiVphWOHXWBMTYImbRRdUKhhYfaZAyHsCugtWioQZmSfZnIzEYuMYrQJEMCVqQutcwJGeoxhHnGHOKDkwxodoVpWWGDQIaXeyWPeFYQeoLOTIBaSPZMlLrnAUTLCINLhwmFxkPbIpcTRyBsUYRsWXsnuHsDuAwXvREJQlFBeTvFzRBEDHggjsYKpcSLslbxIBNOajuwkuLSYBCyOSEezJYfGORaLUzBcJTiRhkScrifDirKyaODpWTYyGSKRtXUKpIlnMyqEwPltmKtdPKOCOdjLHWyDPNpYaqJMXXbydmwyjzoYgHLzZQKCPITETCQwhZjvYosvBCPLMkuUXxdaDsNjpSddOXDQSKWprBusyuMqSaNlTcdATfyqXSszQmOucYhpQvpSWzlVTrkvLcquhlKCclkYbkDALfijCYsSMQVaWSFZCuOomefCLdwjDqMPRiZYGoqacidobZtCyHeCuSkuFasKqcpZbtIbZTHqipLJcBKvtbXVJwDhtVIOeaKuQqQRXPDVVDkTuQcpoIcyEsNfCPmoiNacqXVKRThRvUluxAaKoLuZLPAeXIHRpyBnqzelSxjIwiNiOzjfppCehcyVUjZjYzqvWEXfgpJVKAnhLTvfhzfVJyQXTWRCgvyBcKZlciYdRuuASusWLOKbTGYcZskJwvuRgDLFAGgstlVRhkMQuMKNCliQrGhPbaGiWnnqTNhoSQGcQwWdiMeWYVAvPjQPkDEPktyjofLGvjmAhRjGCCLiMKywkJvtBoLdavZqYkfmYcIrVqeZLCvDOcxkaIoAOFKujXXdFzsnJOJeqvhdEOtcItljyVkwYqJttUIUztICHMJoHgAEXTwcrvqpYpQzYMeCfvjFePIOmbqFapivqimCdcPZyzLecKSolmbhbnQhYkOINJoalVvPcBJxoGDKwGGdiZPoxmUBfSlTqXXPzxNBrguSQwHFHPqWhsFIGWWkGeEKVDlUCUuveCXCLVKuKwjlkBEwKQrBjpFMzJqqQOgnTIgHTOJcQScGqxuvXHLfaKrYMjixfPUlPQVPZLphpHfBIlBhVGDTkifuoTMjRHYInhHxVOGGxzMhtOmwirXKmuaxHUYdplUEUYoHZuEFjeyzTkkbNbXSRUNQfYcPCyNMZKODZTQGXTWMzbdFSQQFTqCJWIAKXBmOJtYyWfdxJnwETQdLVSYymlKPoacfKWpPITSoCnMotqJpWqeoPHqjrqKHQhShDGvaIyOBMoRySZZTnsmDMQpcVdDPYlMAQlkJvvFpzhKbqMPAENEWWYATZULFAxXYqlPSaQekRNRTWCkWLhlPQFVyUnYtiLhECHqrGfYGvFymjgDqMeNPTjtYdXxqkuytmkkByeQefuaJoqffuDRkdfGpzOalIOnorDOSmfbEdrZELKFlWlHVIBgJRprJxzliCzFMgysvoKbuLzrHHmRMKoUcNGECFgOXtKVXMdXyTgsjTjOgOjRntxELdslKPDtGaHWARXJlByVpWKbhgptRJaGMVJDIdhFAjOhVmadrleLCNbFiVwakexjAJaarPAaNOTsEnzhuvvXlKDeiZVMuQzTRjWqyKPrwQbBBeuJKKLpEkyTFahJcWKzkZmOBwPVDdmGdHVmUBNtKGEnIYyNOnoMiYMHvKQmvdUctROuRQvWIZBewyQzAuKNkKOaQbvaequmtHUtUMCyUuIsqwIPwwozfaMAgHAexNkoYHRJYTYxvuJFmmbJBJzvLmDNmPdUBVAXvTgqSopjPSOKSWlFJgHpMRXKIkLBlLqceHPBIzUfNhTqlngMPrgBDDUGjxhgSdWvuKaqOipQJCEduCCEACDCXTOucukHjihYkfHoaYyEZogDecAoNXLQjaTiPxckqEdwYwbAWIKapYzVksHlDRdwnDEnYhHQfHteiKKeuGohlObMxdIssOUDeqzrIbhZuSYWgHDRfBIEsOUjbZvpynrQkWIirOxAuJOqeBBnMjMCXCblknlWKwgLNLxtwxiDVmhABmUyOBgdFBkgIBoquLPeNivUMAxECEkvDCEAHEgnLxlYOONpxHHbsAFutDpIcEXAUHsYRQwazKQmvSIVHPzSHOBvNNqTOvsbLUedOoDEXBZqVsATnRzFdxDurwwnlIJvDOvGMsRjEruWFtjpWkMjVTdXQbAZzsRZpcywuQANOWXUWzHLcmAqumwsXGZOXBlDvTTBOliQhljuVbhzmtDLRqQbtXPVwmeZeTwTvEIhVZYAPecWSnWlBnTUJiSpiYKskrRKNAdLBENRNRYTgTRyFbHnavkBGqRrdkgWuEtVUHCGaIAXJnBOwPKHbKOWtgISdBzxEyyygEhLvDKdRsUAkFGOoZiVOkEMRTsyBiEixbGNBvLNJXuznjYgHFSHsMBFadPtXVtjIUAPhNaRTwCXZFIUCTYjtTKliwZFkqHMOgFsTJpjQtOSHMUFBvcREBRwEpVWZmecYIXVIGBhSESCIdcgCCCEhahAvJAAiKxkzhFlIxGIkRniXgTjqLPkVqnoCqSnfEMMGciFYtiJBMNLMmmQMBcCLXhEKZiwPqaJbgwEPJWAMQmaueEiswxmaFOIUnElQNpfseBUxFuFfNQFSJKpzZyPFPuBJRJzPsqwczciTXEgKlzKbLcVRnIxEooytZRCXeFzKePYEWFVBPwdJrYggsrgiEaIpgjVyztBNVIUaxKSyqIidmERzFcejQYqWxBaGHZMbhZHzQHzjPWuAOkOehsLiqXwgYENrmcJTHURFjMaZQfYVXXctBhDLUObGjDNoDZLvDjxLnYagmpEddMLqNbQHHuVMtaNOoDYtnSkbPqZwQVJHgUTZrbuJfjHRyZBsfTAyWjCbxVilMETWQnBtVfQUmhDxTkNpLOPBziJcwWsfZuVCwuadMwkgqRyZtZFYJlvrDhAcIbzLyNZdbSCmUOODFLSEKtKjCJFHYdgrPikasVmMwVZNWySMULXpHeGpXowZmjRegvcsFoBFwTwhIxazRrebQSnJbYIdZdmLmiLPxlPDoPNhJnRSmuDCHlWhKdfviyStCkvooNZnlakCsdAFKfQHbvDVDBayQhQONpusyQMqfNADmtHCLfMqSzMgcbbKxSQGAqbshWEnBATbXrQsWumuGmcALqDgzdxdsRHRaQTYSspeIRJUpouQPkgRsSSQYzTtnDxcMpcjKVgfYIxvJIhsNkYapGuSqwftSyQWmpDvhMEPolwXtUrCwZxBZLmKThyDQgwyiKxLmHhvbRxIfyrDkxMrLTYtGoUZMIjPZUvqRaWzUkGLkAjxtWnclQLkdkriwRRMvdlnWlUGGDBXpkpLglisxQPpPIExfDWklWIKaDguSyjSyUXHUJHZuykfYOohVKsvDtBWmezTzmEuNjtyYOtlrpJJHqsUgrRMtNWqAmQVmMGzoBLXIifujAZWAtUdFpbvIGwneIbwPjuptRBDQXvACjqBIXyoplZzhzpndJmCSkiZcQDFNGkjPaYVcTsDaTNePqnFjFnRgHHdUWNOFPePpBGjCTPEZdoNGUneQYSvBEiFuqHkkaGSymhkLVtkeZlfEZrWdkKswzWpNYdItLDrGtbfFGXvRtkiWnZXLCDsHUeBYtdduFTqMwzwZtwkWZvZiIwRhjrZcsNnYimkBTQcmQjhYamzFllmNTNhclviqSTUhCyDYnGMOvwBRpxBiNlfixugqkmNKoVTYsVraDJftrFySnBSzsHgsrONhAmOzdHIkQWjWsJrOcXxgfHXipMUVQUKntgDufZHPaZfYBmIhaIuOSoanYIoCtZoKJWiWjDdASqFxOZDKnfRvMJxAeRIEEKDzYTQDLNddVPOLKGxQSfmKBlcvKezHLimJYMqVkTkmylhrmmvmsoMvNuChjXMzvdDdROWBpBhIveKuqqkMVSNzYCHnsNLGoOOdOTFKjYFLnDvLjHzGEwevJlsKDYnruwOsRyGWqgHDTMpqVXYgVheWWxkbxoIrOiKltuMDSZUXockMeTtOczYCvmUYVBeYMLygKNTAiWckKEYPzmYZrsdGEwNYZErcXzlmDniSmdwzoyNHoclfKRhpMRLapDmuSrGFZnHGIxRFxGLVrScIsniMnOdUqNmcXIKvudNoVWgjdRUpDxozYzCCqaFGCTVCkKZxDrkOJvSYlMEHpKJLQDFJLrjhEcAeFFrafMCujjFfsSQnXrkIfqRevxyByfEhRZGGwHUBaxAdoawXBkKpvKhaMnzAmPXypqhQfGqcTTdcqTMmMTFsnKRMflXdPYsIHEApfArlnXvassTeZHiqpqJNKptlqNdbLMSMFUpvEhtCcKhIcJqPXTsNKnOhnrbtIufZHjhiCiebWKoBIHEOmgOQVvQNBnnWqLDZawUMwHaYYrAsBHQWkkywOYzhrnocTnsWuagpbaqnluVUryHECatiRumxehfAfOHdAqiUZildjIFlmYEuVGZxaASqWRZOtgtntrmvinwsLAOwmFlUMhkUcDbGPKJpyiCMFqsRWxTdCgusGmwnyUuoeVskyQSPiTZQoTvSiMGrmsQUfpqGhCHeRbjEkfuCkDawSAcatUavfoYHYkSUFKIJyGJZAYNhJwTWYaUWPdCCEkNKrZxnWqylyWaQweGpyiTrnIYXWoLmTZgUpWTrTtaSsqCpHJVdPjOHmqhyrcZmiloXjjoFPNeDpPohXosbZcoAERIEMGgKJhyDHAepgccYexxlXqpKmtYSUZSkWkkXoeDHRPTWicmHPzIPXfIzTgUuRNgmktnZPmTEJcOVjQhwBXsXokMmyWAieCfQAuljzBSepQcxiWVVIedHmCclcXvGZWXIoLQjYHjQhXtoEAQbCMfpyWovFwKxIzIYuhMGogsHVPLGSlifuzHXGLfuQnuBZFMjAvYCOAnfyxpgiQOIfDNgXaIFtXYoUkNdbwzJBTgTovKlTdMDVEbLzjKaGyoMYYLoGnfgRitpDpqBgwQJNxFkxbefWrccMXQCRrcWtybjzcdhOKLHCXgAUsaifqGUoBHDCtYxFFlDExAcdzwDVxZdbeBsFCcqoxxwvqdgSCzOcvsvSEtbKHhEbPKUEJdBxtNZAFjqJgimXkrPPgslUGXHSgmeyesVQWgoxthcHmOXuEsywFaOcVlRXqGIvsVLvCFRkgOteHcXRbxFczZHHFclijSjBmOlxuhJfZJFFwxKPQbtdeqXLkQtcLRWvQdHrTFODGTnQzUKywRKdnDXiGfdfXNdDcJHvOyCGhQtVfxTGDQSTQeIbXpHxseBQugwZcpTxzAWHErwSZfAivubLBBZBfXUArGpSWyStpOyAMrMACBIBMVLBPlonGIlZTWWBHjbwrGQUSAExYKTFhqJHCADDuzCxTdWGOooQjkJYmmSTWaDHVXARhKTIDpaLJFwWTKyueFgoKXwFPDoKXzbPwzUiGctudLFfubxGIXujEQnUYAIsacmKaqzPgYtDrauGZhlRINQdTVTAZZJAJQWLbsNZWBJNnOnUyeELiXDlWqVclwTvGITvilwhuLYsZgUOfKTxjJJyrGwFWtaIyMNiknetFlVXlKEmGTXQxOCsQwtdHnIECWsFXiJGdnFvjGRemtfVrAbOkYLZJgnPuXyhigUYSFxPuGGQEBuGCPWhLDPbDkQnUxNIotmvqdsmKxzjZLlIyVBdQMuePaZnEybtmrSRzHMBFlZJPHojjpIIwKcOsuKHMEgAQvoErtAWZneteYUpbLstBjbwcYzAKhMfKxiPOfODjmgKahElpaCtNsqDjTkyCkSHoUKRCAtpbzRsqeJSfygLwWNxNEVTOWRJewhtOBFmABtYPDYFZOunBoVepEsRnoXQaHRHoVpTPaKYEwZBTJPHwyjtasenYCiIkjdRHvRktnKZHgHaTXWzccwREFtAaUQioTKSNeSThlYlYivrpRObJLfRwekXXQsJcDZrdbRQKcHQKzvkzyoKbTgBYBbGDhvsSmVUvxqYIgkjdLBDMhUqFDWHPGsjjmKcgHPznWQaHnzBOAcZmEDXXuxQBjMzIMdOtXoMzYQefGuDvHiTsckQkpnXtutPyaePTkQIITuEcnmggzMLTvtOBdQnENpdimkSbkQJwBvLtJCNJNxkeXAcJBINbtSdrlgidzvnOzjpJNynqLUiPNvfiRLPdXSehhNMIEkqzslOaBSsnUhMpmQEGIcpVRVDMcMguAlbgjoZVoWqpUzEMZNHkJgdnLCSqRSwEvKYSyiRzYfdZBNakpZKDmRtOIInrxYBRycFLmFCrnXXscDQtraHMGtKRYMIIEUkEUrFkAKmrFBmHwEsWovuCMbTMuhCLJNNdxpFHzsrFzmJxwribXAVScByFhwsNncDhmxnkureAlzJqGdvsivtNJnUUUyRWCQdemtEjoqbkPkcPyErEQEybxtDNtSLEAyTFZyVOtHzAfmZdnVutjkEyeimTLHwKcSnUaFjVnlLPAXFsnqJWMJtIdhFSXUqunGozcgJHBOCgVdYjyebGzpeZDkFrkwtAYxylOPVEjoxcMtOrRjWqoxJKVKZhazFxqnObCltunpuKySknJqmiihFKpkWxsltRHZujQWznQVPXCHYVxmQWPlvHNdEaRvCsmCaghKYeueDfngbBahuVkpXqkEekrnzuggRMXFWHFVUuYdAvbnTzTjCJuceEMaBuQmbbbzolKKaUEXowwWshOvVHMPChfpkciNYDjzvIcWRyxaUuQBwSZYLCgcCentwCXUTldJHziUiwTAptgOPQBXrgDJmclRaoHRskCGMCaabXJVAgsOZhWGYCNwDcSQcumVdIBmDowHQUIOOrRhqMWaeVjVzblXtdEqiGoRTWtBLqIXOkkUbsncjbrfEqXrYYMIyWMKctFnWOtAgjSBYJDTbLInFMoJPDJcTejqZJtTyGaNbxSkZEzISNfVTpTKGqXwpdiiwVQZQrVLBEBsHamjwgvdjZqJTqlBnsUZsbvDfCRDcTgkWYiUTLKBpGqiQNTwLYFSWoiyYRXhebbaVdaNxOhzKgLQlDlPfHKHjNBcdJfOYkSEQFvzGWXQwKJaZceCHYAfLXyihCjpliHJsxHvXzbZqeSieTOTYtWlxyaRafgVTgFjzljXmngEkKgBAMLQswDGUAvQuhuBDVdGGSYVuVMwPsjHyvLEYJdBlAOyXDQtLItWrtORFnxJSdkUPkrClKdUjIacilxLvsOQxiTBjIoEovNrzGAtgOandYDzjZUHJiYrmBWcoUnBkIFxDSOrhhrBulQcxmhavZiHXVGwqnYLaHuuHbQxLZIuMHCRugrMpKLLggPEZlJCkXvGGIubHSFFwCIHouXmpNbGNvQYDKIaoSWCACsvToRlVrhiZZrIcBmTOCbSuIHcSYDojREgewxessHupdbLSpbDiwPcGDVTEwSVlAKjTCVWISXqbFkVbesErJkEbPPMWrjbsjIsMmbzPVkfsfOuHWWOHDWwbYwhSfitRLElfhzZXqTJxLoBbuzYAuJGwGSYliKfmSMNqNtnmnNFikRoCeYicZpSeSxiNmUrXmODHdgpfXFCRPjLQjnZecglBXqewZOHOgMOagRZVJEbMkkUDQjKHIadvxSyBKIbGLmlWvfazGAmHzaSbOTpydxfKqvWLqTnnOKZfxiVGMGbTjkkzjdPhqAeinXtCcpHrpKorfZRXJjMohajLRSQcIhiyXwJKRqQUKJAVmPiCgaxDsSikfGATURMHeRumZHiqAQbPcyDxIZgRiZowNJDqhJCWERjttjFOnLCJtpEbYDscNptaiYqDQxUAWwtGCEiUjKUYbimmnfBPcsgFHAsFonpaCrdNDuwStEfFkMfRhptXDWIeDOykzIFNZSMnvELVhJIylUBvviSZsVEGNGVzIWzwtfOfcPXoqthBFhJLOxLAZCdUWXBEmWfpKipEDibAuHxmNTBlfKVDMVoFFHMuPPoGmThQAqVGPAxJtERWWbKcvbHIaenKCTqwjEtVBJyXEntexjdjxTZNsGFAtLCFuPJaZUkGUorVYexKERfMtPSCBAUKRIzOqhFXCclQIRLePfJokQBtyngfzTmNJqpentbllfrzPAqCbBkfTKwLlOvhrgbqsGvfGWxImvXLjFGRZYXngppNMGyCgeCSRaslSINvOMxDOGslEoQiiKGXhIYjvEHpwERgflGOZEeOiKlTOLPsvFdvElcQsvPfReWcXhJZitisDwxaxhrQJjQkrMWpbfosOgiOeSdkgTTwfQlEdzBTQnEgfxCXQXgrCiGQkPMzmCxFfLLMglkofuEqOKTsSdPzKgUhmqtPTrhrfpfBLcUTkFSdjmEqfnvqrxAOVATVVNkEhKGdRcOcQektnYEUqtDdNAlAkvrDDNKZxkISmxnUwJzAcPfGkDMvOmhIRfzbjdmkQXeLmaiazdoHQwYibNHlcSKHjBQfxpVMAZLVaZBgnBfBTUVwoEjUKPCozzpbABUuCRpcALwkKJUTRQFURdAlyCJeMEhowkaGniIywvwZkPYzskXUZKUsceXuuRvAvnHOtkMqlQqopdmxCcwNxuXQVnIPnVUgmIoKXytNuPeOnMycUWzCKExrBpLpGjGHXHTnsBlQprHnflaFNDceOpcjQpPjphOfAxKuPEgjTpzuysgdJElrqJhdSlNETylHsSBxJejYmlFxPBnpjQfPflMpslslquezeFNVYQmDCSYiHFUtwGlqsHlsJjRSPheMTnQufEtdfgFwkPRsuzyBEPhIRpVVVoJSBREZxIvFlFAfJfmgKEMwZbQukoDYiLzunQReuvoItIxvIpEbWgHoOuubqItvCWzGCXQrtnBVMTTBmDzZfpuTOjnNXDTDWbhnDgDUrxttJPVJiQqvJqwsvmITVRNlvjUjaHgyDJmiATtFYOInYaaEwUHLBGonIxWCsTlqNIglyoJIUUEMscldoLATQFXGAcBdxrCQLxLMLyVWTIsAeupkofEOaRABvYZLntIhBFZTDXEFpHpNccCVbResrXFkMOWGzIMnYblgtarJBNTViXQgYxtcszBhjTynZXfUBJHNATIOUsNeiiFIwpimTUqixXRmybkDFXlhKhrCHFMFeXPwcWlcjodghdfPWvCLyoUpgXDRZuzIvilAfQnvMfBNoIPHYvjQhhLKXuFKbCEyTJUdjkzFsTFsoZhAgnfuMKyhCfjdwOZnDESvCldBpduWXAaLlutCPXywRHutGYnbkDAYzQdnvolmhjvhsXUalyLrhhSCXeULYFOELFLWFiiBQFbfPSpByRlDNJgCkakwdvOzQqiqepOplJrdZYpSSApaLCPnhJFdujVMWnHsfpYKiEwVPicKNeOprSydPSDZBJerLrvENzkvScavUDYDSEhhWAzNrSTUILEGvkABSfUzXzZDAeQFRwHPcGPUsMmFrqjznMnfLhOQNxDEFgkzhxpPMGgqiIASTxQzzroPTYUnfVBnOoLfBvstojukfeWhjBfplESZfVmKLUswxQuhbGQsfuraZeQRBQkqrPfXIxJKJbBoirlYPxWOLPdjLQjssozwaLMSKlzZNEANbKhobXqsYfvvGHOSDtGEQVIwjMbvUcgvDkjifpDGLiNryJdKHEfPXPYEkDgrABSXPwHhrndyOwbWuepzWuzrdqNyqAvxgNdaerDyUxOmhknDuNoqQsRoNQWnoUttxxNsesQLNplBpjOFpQRIYAPvpzioAyreTuNiLAtdEbmbiUjrSTblgOjhjCGmzGgYhICdsBSOeynaceWpyakjVgWRikNcYXfrHNmwOzDvRjWtecGWzymZXIMZzTTCquuUHJXAPjoKuuixWpsojURLHzOpwQdRCutXohZHgrkrrUSOqaKjOqQdCxkPSswrJIzxhxAXdguqmUQEtlffluGsIsWCLUUVaqhMCTyqOtRniHSxmrUswCsbZYMfEvavDcgQTICCpLSZmRIlNjdMAnMivLhIFXxQkABRMVAzgzqJqKPuFxFpIxEoRAlaFosJdHsGxjgObqMLaCaaBqwFeuIHJgcTgqEyyNbTwONkXVHMKLutXuKVDZGffYmVtIOeTETHtPRueDAiXXjhmslhXZzsgRqoibbhqKHniVZpyaciRqzeCSFUHKCCIjlGJHyXfUVuwrjZqmbubuSSPVeosPVBckbjYQISsOERiJCaQyojRkprNXnoBThUsNsobyMsaTBUoaIOIpvBeivNQEltrdxMojIEgcZcjCmOqGMTOWzqjGsBSkuCigdpdBsMruPCDaOmtHNjdrpepWrCvKMuJfDODFdBFffTCOuNxcERcpMebBluKQFwRFYsYXFSTlcapbBAzWDFbwbCnzjdCZRuNPEcCHUMzmrgcEFVUgZHOkYBvIqLkvYuONqkMuaNzcrZjApdCspTJBHAiWqffygYiVoTeDBkRALZtFhkJSpOFeNayiTxUVSupdNZONAbVEnLDfWErpSuEvFBkfXLrrEaCNguRjPBbaGlAbVKNCyrrwwFXaGVzFWaQpWPsVYjUleYmkyAOLhJPJqXOadjVqyeLuxPKdcopJYWzGuoymtmlrZDiDopbafGyncODgUFjDcczOdFeCZVTUbTipehwwaRDnQhHEvNZmcmmhhxJfpOnqCHZpEDiiSqzgDmODkQNRcYPjELVmfytQWHaPxEKIoQxfKfbnuGHOCNvrYcwWSKkbtNZiuMOpVWhicfcocGrsUJwQjShjiVJLqDauZTkxhwJModgDQFBHWNBhOwDKdcrJQpVVVorvQofpSUREjmPHUScprwBEttYFcdiLSqufDVKFZoyUfagDrraxXVWRRqikvCvCHufNPdZegmRakvKbvGXbpNHEbdNOivUTdzyrjvhmpXtfwUgrYjEKZYfEAqQdPLMgoecPTYnULuIgTYrARQBjepLALKmPxLtGjSocUBKCOmaIlRVebTQfpMzUUEyledprGFBuJweSIitbFLVXyvvYlNIpwHVLSfrNQwCbzuDZDNpjoEkDBqknSRGoGjSXMsrCeEvCJtpvvHclFgtRuXADZRDzCxbKBhdAjsBuhbWnAZuBPAtgoYJKIpsKRuhIFZDqXwLSoUTgAYjsRMQnWiZhOTJdCpgCQJmzWbFqMnjgcaNVXrRpFvHZaITiwOHvfFjKzdEMLRvczUWZjhnNiZWIyuefzsUgQfyNorCfvxELRRmYAhHVzaAUVbNrasnXSVlTFltIHgWbYvmIJQqrZCaFHvzZoJbzoxVeEWVRqztpiSqmfFjwZszZWDBEDGFxHVhCYTLyykEVGzgiwLKHjBgzOsCTUoXmGoHHdlyyFjTQXjwXqQStdPyUluyKJyOoLQVTqSlcaBEmJnbhzzxeRAmGLtIPiXRXiYoCZpQxPHNBWxaUlqwgFsnSgsGXsZirOAshRdcgYADRhDTrgKPUMtPyYBtXVNiRuLDURXrooOINDuKkIfeVZgAHkQOQiGJVEgsNMYosYveiGCNbzFKUvSAVlbNUQRSijqQHMcYGbJdAWReevrPjnPIqlVxgEvRGZJppYgmZkyBfVVXfLLzVukzmsALGEmpHwFnKJMNvhDCUGYajWSgGTDwPLBskpkGAClbHkXNgPmrMcgSqCBOllsEmUkGyDaVNyVrNNAQyjfFPWXwvSpMxYnmPSygkshGLbUwXnxdPIWmcEEupacQGSbdhbhoIRVIpylGBMHWmQQAiypIxGvXvvuTLWqkwUnioMiTSWKujGTGnseolTtRgVpyiAPWXfGbrpaEYyAIHGQePeiLQKbCMQKiHqokhbLuDnInnNzRKxfvSzyyJJKzciveghXtUBRidueJJOTBtfsKQHBDFKsIpshjLOfpzxEFFBHqkJddntzeUIHvkmqzyfazyQyFEdKxUfFWKSOJeoqDjSoLaOrUejHaIjrGoBslujkrbGdptvAtlVvRYxhAuhmePRKmLbAVauctmqLLBekBtJcbkhBYiSrnkfNKlPNounIzSHOYlPESZkkmUpcvyYIvTWVjQXJeYdjXchUBqGueseTwrVzOWfBcorARqmQWCoccwErPqYnYeHvBEbinHazhsDCkzCDqkOVMujoswIGhfbmkmzIwqkTEUfeEjTSQOpRMMuaiWVJfNlIDwyuutkLNCnwYjqoPOUCVdXDGHJAIetgdDKvfTldbfTpPjyuhdnKLJdqCxTMpqCGbwFBKXbXwAgjYlVNjkgtStQEZojVNJOoVPPQUCqFKSBSVmROJtnzBfMihFdokSiBMwapEELMYdxPHtslBWEoMBLOMTkamYNWZwTkfCEtHqEFwycWHAPRXtbgoXjlHlNAbyzDIqJnHZslbuzDOVesvcgQmcDobaQjGHMZxvtMHEReAHlytdtIEBIxABxYbCumwSVhxjWaQLwnxxWakTloTJeHUpkXvPSSXBvlLVReVNOJMffHQGKLABKZhWosrbvlkyFmcOwufdLMDfZDtILAqwnOAALySGgsXZRIaHPqOqYPSndyBWgkSvFDyKHgbBxcBZGfkqNKwCcRBhSlEBwfrLCLVXzXhfimnTvqTfPlaFcTEwlaZXAdFLnIKkXcgnMdPNjBpbHcVIcTSWVQJsLmQBjfXjjEAQtdBzupOuZrwvxdlWHJhEKWWawNMsHkoPlrbhpXoBudfAwoYbnSapxJMeSfXLIROhjMTQfEbNFUazkWBYRxsfsXtptwHIupNbBLzDnIxshNXdPdZSSACCKpSRhEpUBYQUPdirWlhrifhURmLapDkqTtrKQSnsPqKPDxfDVzQhLKFaQvFGXksofwzhvXbiysLrQdWipDDGtSonUUHlODgCHgNEwuBqnBRjNomAWZYMQVRkubHcjctUfOfiNLTuQcYZcviCLNGAnKVzaDyYDAgiWnTBwVkRbiQuHSWGJBGirZRTdTmqXilTuZKwoCGMhPJftaJxzMqTJJlUACvCuuChQDNvhKXHEFCAscHqijptcMvLhFQKsNzQuhZVYtJELHVxNxfbGdVFMdZJxrQALccTnQwMLBWUwHfEDQqsxzVhEhCmBYPfKMictTHbgEYOMoRRxqMcYwCuwRFOYnYMFVZkVxfNmxBMByQxcaUTnHYLCfoUJwJUGiIAzqgIwvNUviZYGgeaODoROfVgepJjEIUPvNJQVISwYrppNNWvzWfSHlGffGMIFvHXUrNCGbmDRFIvJzjTVbYNFovcNlJzhWmAaKEjKbfgSFTmNefpFYNoNJXPxzuROimDymDvKqJKMycehEUcBonAAmAOvSWOscIZSuGskexPQixpasxtEhQATdYlpVzwvSZDqIPYeOztrljNsayjPKxyQjwkacVjwqjHfkkhPNZLssUUeZXtpwAKdSxPOJEvEaFTzNhIgOTUQfZNCSBmrjPyVVEslWVzipJTZpBlxYVPpZUOyPdgLjPgQhufQpfZxkTiXGsGREAYUJYYmiBmweITFEcJbXEUJgpmNNWgTnIleOeQQXgvANBVRtvsVpIEDjdOpCBHsNqggpbqkUhgjlnIstyKqCssREqbGTHApVQBXQvncAjsHuWTMNExFvpafiMtYBcISTOOOpHZwYXfrwpnrTPeWuMscopqZfxRiKllwmuDlrbTmudgokVTzgZJAuUubEFkYdNMUEWGuUmtlPZLmQkAObfBupGUVOdVkXiRWwHldjYWUzqbEpTIqlIEaLYtYewWZpbJyCulHENgcJWkFYoKjFCPYzZFCkbyAqAEhFUnVSRnRQEfqaAYONjzVKtSxFSpoWxfulytsVHuhaGjAKQGlvGYGKOsHOdgorJxoxmQGbOGggQgEzhLbuxZFAiRjybrBSioWdelqkogUbINUuhTlbSRUrQEoxXyLjPrOhHoOycNpbFkpKwVywvbRpNzLzJOAkPksnKGGapOQwayocosQCOhfQqpWdZlDwHFWWKBCwFSfFXHSnhUhJZgCaeIaErwISfUsNmzXrXkhGfBIwJUzhWTboQVRrhgXZwAhxDvfbqHDjEGhFgSsOFYkjRUucSutpzkjUcwcCvXCsaAdSrgTKDMPSnOnYzRawewwwUnCbDZhGMNPYsCWjFyjplgAcvKRupyYpEDUrTzahhkBopHCfsprenchMJlGFmJwrtcqYUFLxTuVnzuJnLYgFGPRqUZdqebrciiFnnqUvZPPACKDkqEBxtkRsXaSOsKSpIpAAwLovpXBJeujvWyGCFroiaFIjNdiDeidoWQQLwMyPNIeTkYRdfNzWMtTTuddLvITRCVexzbEwUgxvFrPLuFKOUvSPdbiZAprdmYxyoobURSDrzThBUzNDsrWaTBqyWKJeiyykrwRGfzuUrHUMPfCeUnivMDIGUlXaSOzmifoTXHTwSfkiAoibCZpBziJybbeRMTypxVbxdAMpmSHMFXfhpavUrwBLpqTPGpTKhjEePLzNwQWSeIAzHITUYXeekfBjDWZgmANbzDPRSgrCYmZCWtufUMRNRYimwTwbJBxJyXIvfehgKviHkALZiSEKcEBUoSWYuxFJupnvBLQIBeCnDQullLDXyfDqmqnKmXbyOgMmWSRbHNSaYLyPYPmHKWsWEnFknLzUEOQZrZLdetkUklzKqvQgEjMBPCdQGQCmVlpyOajENQjxPpQlfatHqteTRBsvliQusEmTBbFDnNANMMFjcIwyoIHWjFpAtEKtxBOFPFRYPAFGLjqmoCFWlYEQhAsCgLPtTlIKGjavBGqdjLjePgWNmbnWdtLdCsJLHPoIHMymdZSIwaJEswogYAygOZeYptSRkabEPqFBPbSJKmKRIKsLzItUSEmXVVpqICwujxIgQvMPMuqWKVRYdIrYBSrKxYLfniNdakDWosKKRtQkFsCBXNRsriIGGvoyUyfoDeuKIfQKIKaHLzeBNltktxyRkzDIraYdeTKdJzBljQeYsZfYKiRlpkgQkQQuvHEleKPniXupquWlbSlNyifgAidrHsyFjTgkxZCKbbspONizZssyWkgrBQAGQSBAwwfwTIDGbzqJvoNflOlvmIthdyTSIjYRroJStNiajklItIAXmrAVwSTxpqypbTdFwzoQUSiwNDktHYhZDwlsedaSEewDzkiVluHIfWnOiTAfEGfeDtrjPcDQVPkTMejSoCpQSCPsxDFJccvjvqryhbTaIQOisrUtSPyllHWELeEjLXDgFpNFHsjsdXtaJhqjvJshSnqfRRIYZNGZSQTYGtcKkEGELHQWyStLLiGlbXCbqaYrDZmUCJhYcWIAWEUzOnyjfIAyWjtahcaTRaNltaYTKRFJZxnUuODrChVTaCxAMJmeqgcAqbdOjwquAWrMgfuYnThREVPKMYGDvXSrMBoNGuuCuqPORQwgFRWPryWBQUOnVUsiSFWHRUAiOQjyPGUirrQJQRhJkzYrZnPhjCfqSkBbMnkruHlFCoqPlzuNUNARVIFbhkgBPmurepOwKvbgNksMcUapYLkJHjVqLoQIlVfqDOiHXqSHoWlOtuwmKZdNVgewEtVRxQsyGYHRfFgoyIGtNxSdVwQJEnsewLYrkcvlFAvkguUvTInnPlcKGISnLvdrSOEcZZPkJWAwodcgfKQWPSbMZcEJrikgnbLWIDAgfKWVUsqTieAHkTnRpudLXVxpxyjyZUPxfUPjveKwBwctUJSTYBwZBMsqdkAfpgEyVQYENNqJVmqaxHzEAgSdCddiMfYsVxPvdcYtabHXNyXIZOQnDvxIfVOFYkDUYhvuqqYFoESNAVbprVfqoVOhZHSKfpGfUniCexEeQyLQUJcofHoqiarAIYxqtqOfHqWStNfCpiTPxAHAxMQgPajTMGZlQcjwCdCMPZDGvsKmNqrupPtyrGehjepNJQdLyzCjYyJVLklOwmPBUiWcNofyfZILuszrgBZhguhwpJwPJIMtwDCmrAeGyczggjtLPUeDGyaNRHtUfGmgCVUoLxAICHIfbEFRvoICgotXIaFFfktwZwpHRSnzCqKciEjmtGByhYhgFkOBzZOqDWavkgQPHKpAWLVjPZCnUikRIiMJIEfevwEHLFOcZyemnEwLgHxibVDEjJHXlUvuVgEBXerkKrUfbpTBBloakZqBGVxxaxlUmAhLSOCOoWqxXphcQoKWHWTnpAsVWvNjYeJJllWqrSFifwcpmeIeATvcpBLzhhFPGhkGRxDjiPyDWWVBVdFbfKmjjKKEUmhpGtaOawvxgASxRitDlSjNNuAvNHCiSTocmdBRbvRyYjSEHDTRtKCVrnUxJbCWxLWOxQDuRETABsbVslcGlgqttQbHGiYcnNtyAaQEHFLaZmSPZFZyjSStqkhkXZBhtJTsgCueLZbgYOaDZfkcHfkSKfNLPTRibtzbqWnJXUHMjTMVyPEwhEXmVnOdXMGdaJFWLgqEdtXUDBgLmCfzmOPDhasIQPfAZciTelpdDNmyTYbxDulHokeSzBsMRBRKWWeBWBTAzcsFPNVuHStJfXnsxYqZRbfWAIvwkuuAVTIjjCybEyoGQevojJxCHKuUwQPMYBwbHJwmRVFktPKdRaQSOrXWHXbVIILmjgeZpPRuJQfJvDoEFSQzppWmNgPiESNcMSmdstAuGqFmKYGfcgIVbFLLvZtPnKAxhqEeIemgPxffLcYjsyBXhrczomyZSlEwvvkdelfwSXTrqdQoYHgaPvaVnbvEqHwKlOWxwgudvsMtglyBlPyXUmkjiFKxmKsooyNTqMJQRjbOcrheywvGZxDERVTBzNSekbUREmwCUGDMRSXGxkWDmAmUkYaPSNyUFYXNzkbudeClkAfwcnccfhghtuZHDkmCHziEdPhHYKERzLofQDfBiowEFfaiwChGhHvNHzQaZEnjuJAyxkaUmNXHvKDZqBwHBRSqHBzEjjjGJrizAdDfQQquYcEFChMPLtSWUHSXXzQlwyWXVWcXMBqpOjuWZqcUMeKyvJiaqqlnfQWVZxlyYXPHCYfsmwxaCXigQererQPRGjUHQtkFnuvsdrfuQPnrIxLsUqVZwHYRKuLNZgKarsiaGNIFFctYhZhouLSgurGaSJjCelPKFLrdLDbDZJQqIYcfcaFzKuYwetsGbqWlfnJzSSBNUAXMsIdOopiDARLtjcwfnSZmXEJSjJoXdbysrZQupLNXypFLJbaumEoUvfBregaqGqrRQVPNnKlSgwbytkXEYVFvDmFwSggaATbXwquUnoZpLHSeswqDstusShZxxBkZfjzXjJpUVjKBHTWocyhzUYMbfXuUYhgqgxnYppiKCAMhLxoDYTzzNHBVLdiwKCEEWyjPiPwjSZKhMlGLAsLoTWlmzqMgEZduTRzEsXuXgdTSZzJSzreSfggUNEWngZERFNEdsebFlYWVnLprXKbLtyOlXDqFpnovedtXdBDqHagAhGcktydSlmHuujfxfiTEzmWQFbZMcdCtNWdPOspDZuthrpQaXUHSStsGcEmlgAeYpICMDmegkcJQmHBCgVGPxudOyirGtHOujyDRdfKhWOztEjRyCAItScLevDvifEyPUGrwGGBLprhmPJmpBFYKaqfRYQapmnXLcFOIrihmVsijPxmGAYgKqJSSaydFnuKeWzvgGMGQkNfcOgIbEiUBThjwobbLcIGqAJGebsOGslgLpQMntCnOKoWIWlaCAAJzCvvIaHpmfGaDecpqJgNHqdMlUCtOhirctIIpqwyybkZyjMCOinqqCLuuPEtlMmlhFaCyNmmEEVpRhyMbxLnjdsAlOYLEWhzDaAHRsLirukteXaMZBaAnFrMfeKycOAqNLiIumEGlrKOBLHSoMpTcQFzAmydyxrZaRxLQEeOFOWCSqgOEhuBfQaPmFzaoNFGtoJCrSiTMVyFdiWSbMoOOZRSgXFzxsCmasSYycnckvAZLsiXumWNQbaYRlIDsgtOpHHVKxJBrWaZXBOezLrnUegudOLMvYSptrjWOsQzGgffyRMWPlFdPGMkXMrsIwpqderrFkEmuTBARfTmomlAYMoRubTMXcSkGTLkvCZafmDUEgnmaeOigUYLtidWhwLoWnoJsgzQVgodcmkGYkVZQaDlXgAAYeiyjhkXcUtpHapEAAsMlJWMtoPnwJayIfMwbGQPVjonjbKRhWEkXTgJZuRtKKNWelzLoxkICCbiQcLcKLUKSIJcRznMbHRKnbbQJzgAWZvEQdnwiEbfZjSnUwgenbvRQxRzlFHTPJVhyFsHdTexntRVxMNWZrzcvUGvsobtbshRhoAkkyJSeyIMsDjSgPerUaFArZvJCqTkrfJXlVmscuItALqrttgkVjMtnDVlxhKCczwxHpnweRFNJsMpHbYeuwqyBojPUhjGBXnXLlBAyrHkZEMfnjqfQHhgRSBEWKyaBJTODiDRMGKYXgzQGsDbFROgVdEkKXMRXjjsLCisDHReJqqlMBuvheykYsfpNauMXlCFfQpxdjZTtTmKsbZwsgVrLEvtUKXtnbmjtasXoiZeoppSLvhdsVWsdKSraXFttulHHVCluvDyTbhrIyGEfpKKhUoRSUkbJPDwUiajXOkBpmSlKiGVSomrmwuByYqYYrSmeBfJCMDXQGJMiniVdcAwEdKXxNvlkMsCiXwCRwEncYiSOkiYRwhQfHWZiCckruhYUAjmQthvCCuYBFXqrEkNJwyNkxMoBBXUyQSCfObPeAMsPeMDquPVuaFerUdouyLaqOanfYsrVsvFLjvxycofXEFHqoTGlFXglfltCvHdbCzUIOyGPKCKPgnDFTViaNOyQkOhoDkoNSayFiVwwBRPLmtxHVxpSkSnAAeUpTOoEdgYatmKsMemWNgMOlKgeJIJVHXnIrruOHnzbtLENEKGcyECdCZOfEQGwIHcmBSsPquxRgfztFfSiCnSrlVAbwFlPQtOqZbOsJtCMaWrrRGgxocPAyguVqkPojgXqEwSPESLZPqByebzrzraeMcuMgKvXotwkDbyymkQtMmnhUePSpnuXLUUzoVhHcWfILuBeVgngJUfjxHUNdiMRWDcdbqHETnTqcVAtUtUKHJRMORUJaHdTwzeWNKoPHyAdAyMLsPCqHtCBRbknPKuNGmvtzDmivYoaGJrKMkvroqRXsDhBoquOfvRUCStXfzftNBPCCtlfZSsKqBCtwhMiQjQPHjORRYoXeqdLMxGxTKNMqdQcEbHVHrBvbolCYPXzUHPXyUfudXOMWgnLMVovzWIzBOGiyjrOKitQxlHFAGiUBbDHaTbVKvuyoKbnrWybBqgfCnPdTGCxzbUCaCALjKgGduDDGQvymHCyfTsdqyrpDIrnSDVaKyHceaSixwslZrKxcYDAdFchTlbLIwsEBVwULHhCPAGjFGTFKsDrfgsYCsYpVVhvaGvMBAQbIZpsXaUUFADQAOaDxiuIVmlogtHlTjTjLKVKNbQlPaiVYSwxZNswpzRmUWeSxQsdPNJlznPVdtoHpCbJNLdGaKfFEGbQjhkstQDJBpJVwKZOFnVuYgtKSSDIVdMeNuFJJRaVfjegJHIndswDYTQPBaIiyBDbFkuJClyRENKEVAWJVGAHhtsLbPzlxqEutrmRQEQDukgjxCSKDVovwvisqQarrfZrsrmxEKgNAVmvxvdeJYJJLvhHdLbQGfaGssJncKEuqkcEBgphedgTbstvWyIjsuplZwjvTeeecHEvSHybcdmEehaMcZeNjnyGfymnMMhoGdJJMGCClSWchMyEWyqVcbyYipNEZBhPtdphzGnfGyzPALsDfgPSebGcByNDuwZgtIYKEHzkNSMILyTWJndGabZkeVCFqyXRRFykpGosKQYJMKTpmBVHWeqUHfZDpHQtyzWVJAHWwUotRCFkcDYRHIInXzJCsSsQVgIpxjLJoTJfQonZbuzUOhpxYCoqPdYGQAyvoRbCbVCpLWRIKvGdKYlvLLsQSvyKYszJdvFTtNbFLFGrXohJVKvoIctHxPdZVflWFGdKaUSaPpMIUlvAmOkFJaTmjaoyozRjrHRRcOQbtBVTXxkZFzKlVVeKfOgUBeoogPIQZJmoOkYywsHvciDkYfRQZqIkGlpysMLkFwamQMDDbLJxYvZuNlNMitWdbtPsDvkVzPiDPlWcoLyZbxtpjYvHGAQorgxgpkxTPGhYjEzFrYBTHVJNiltffDGvpQZzhrmXIteocsKaxCJcZmLXZqGtmVzMqOMBAldLkkhhlBXAnJLIefXsDHXNxIBYPQssTVLcPPRGGNVLXmJbvcADhkEKNGxFzAAEXvtksjDPFrAlxwFarsrpzvdQyfCEyWqgBzWDZAPskeOTBPuqhhqiOdpaqCbucOvBZeERmwwsHWjyjjsGfaOczIDRvAdFDAnOcOJaYxDzsoHIBRGdtHsOoumWmBRdYqQiZCayUvtzMXCcxskpSBzkJMHlpzFDNNEbkkmuvWwcuZbkCrMRKEDWCQsqPfvOCuhKRLfeoLISuAheRWShwtwfZpIAGYRYBNtbHJlwVjdWbWKiJCRREFkhQMBANvXuWkKcIAdGwrCjKMppBGCCbKLzxeKycchjZZMIOjPeHALxwiqDYkxLFgPMWNBDSMxbZWyauxOCzzaHrneoPqDgDwVFwcMkyWgzrYbXrQcvIiXUONXNjtLBcGclvwTfrElvAZxxKZQlLoRZFVCpDfTzaPKjiPLxFJqnlEYnfmzOQHHedTxtCyXUjGrohrwVHQEMopdVtEHCmRkzUxgxRNdXLCtwvgUXYDfcOexbfcMLShqRRRJwgXjXcDywVOAHMblLeyoLlgfljdcYJeVpJVKpsxxlhYHfxjNRicnXTPCteEMXsgflMyyBhkNBTThbdYgtMkHfPWZNusXUSGhDCyahEWoZLBYAsoWRURAdLWrexSqaCRqRfpjKwzdSNUShKBddjVEJrHNbjBQVePnqjknrlYbdBgphEcosFmsdqyKFLOUSjKmqliLIqsqfVJUQUP</t>
-  </si>
-  <si>
-    <t>bgCvnVYemLKWJdNZEzIOgbsMaspHtYFAtBiigMjypUMaYqkLgzNNMJeXaHxomPElwPvESxcQGRgbvvbrfKvuqccxqDglTexwRgLpsAzODEAgXTEpmtnhbRbQxCNyJomCHSPZoQbAcsDXNaPFuxBBfRgnjjEeYWzUYQexazaBeaTiTDGJOxnoySQlmPzOnJtQQGrCFgTjNIuJLeIxhqCEjsmNOTxFPuEEoPkXdmvmwPqUUyyjCMTgNAdiHBnKDjQscYUbKqZONSfVnVLdeCZgSNbdacHHaHhUJdgsnxxJjvcRlQxwkxpsyNgqCGYoFYiEljPGLcIjMYcGBoiYmXoSpdbogsbvBafTjxIvTQyEykMCpNKzkKDWIaCxYJnqCDIOTieEeoSAophtwKYPzbmvdcZbqQXdrRlKlXPbGgubwmJQrxQwhYifDgjwsYnwpIlHfaQmQgYWINaZNtQzJqssznfjabBrvauRCzNoeKOmisnEZwKxbOxqyYegKGbVmTGlPpgWpjmNyfLHzECXWDFcmFMEuXWQQgFfUAsTyEwzEsooDZmeMmnVVOeouyPToFVeqDnJujuGzRHSXNcuHGmfXhYEGVnVMhBUvvRjMkRjqMCSMeqPuFhBZOVuBAfMlKgCgrxmuqyMKwOVGQilUZXdEkhTLiMvwdkDnjywTEzECigLaIBcHzPuKKUQcHZmnTTZmXLzQdIjvtFRlecfQDIMWtCgxwGlOqYMXCQnmGhnqodOfJWmHxvJCCjOjAMVQGjHKvxSArMWZqxRxcpUfwOpHqqfQTqwzpKygPGxBclgBWLxlxkevWhuLRenqilukBGzSGabnkjXARfvTbQXoecLECFMZfrCvuvfQoywRTxRIDuoaDvKqjvpBFkQPFykVQvTYcNwPrAgzWdistmCmdQsRRgoEarxrJPLFwMROhfAgMPQqPiZXtZXQmhoJbnwlwymQiZuCnrJILBDBNEMCEJYlABhrHMyVIUcXvdpnXqJkDKNzsqSdTtYOmOcDfyrNXvhsmqksOCFltkemxnqBVhdtKgfIDaqwRYFCmIktlpGSJGikuEZceUlCXcsBeAUwrDCidkMWPqYsIxINHFGtASNrLjAeujIkghbICsDAEiLfqucYuwIbxBvymestoEdYCuOpeiiTynlUyWKxYvnrtLRyizbYQZiHgTOpknmWJZpwyhWDHhemcNJmxIcELjWzyTQYReclwojzkVMqodPCGTSvOZASTxfdoZFSbjboOUvqobauDuRRrkxXrbSsakRbmspIPpTGwTGAvbzIWuLWuEAhqprLSmlNhnYXRMAleIgzdgtlWCZCPAOybUhOpmoVubWtfQApWILQaIDzwRhrdSZOtikbmxHdMLBwxpUsiqQJUxJepvOfnwwIzvFPlsNilaNqpJktJhjHzZyyPilOUPgzSgGutqLPInaqQNVrXZloAEIUZbzYsOBTQewbgxyeAyTBZdNKfzjozUspICgpYpNmryEIFAhItzULsjViXOCArPSmaNxNUaRtktgnegBqAEseZepRRhMhuQwHefyMZwGNVmRZmGjwrDFKkJctlhzjNPQFaoeCvSppzUdzvJyENsYKRWRMjAFDxdOdaCkngIlJbSuFPwfxCDPDVDBkMUwGXTZwCfQaCSXypAFQICJpGTfpfqPVGMeSyVyanehjjdZWBwnkEyXXHiqpfKSoOWELjqgMfCMNRzJVSxQOwlKheShehPjteMRCgXdpiYLkGqsEiLWbkAzEUiiLagBBNxivlUbtfFFfcckMgCTQiwJddkuIpLUTMnhcyPCNTzRWiaOgbfZGNRSVcXAntKAVRTjEyzCZctTjwjjIwtDuJDxwdiFgEiKZkNIbgkKIgdAGgPBRINspgdEyNHZJySOYczaDkSndAwjBoBzvoFkHQrgHNiuwFZyhtfcNQeMjMHYUrnpZaLJnUwhxCsabpPfyEzHsPCucZexWQjhdsLzQAcXqkFCBDSfJAzGIFGzLYlncQZDiFvogkcJYsZdRcjMGmRXanxqyJgKYXymPBRqnnWUQdCQLXAoKzihNlaaOsnoDuDaiSJKqBYbAJDRIPCQdkDkkWSwtRCpBEnUkoIQCucgisaesumlmxPfDdkLScIhJnDbETgXOqduoqJdiEOMAUBVFZIjynwGZoMXgPEJypXoEnmPiQTXPEbZRDEEsMxFapCVCLIXNuyBBiRxCRZQZOAvGdSINaRCRHMewGxbBbCzkJMIFBmaXYbQItVoBCKjkJcwIKKxqEXAwgkyRcTEffqVKZayZyiLUjOWkdfJjpWetiaISWKwjlfxSTryWCxNKjpLEmzoWNWNhwrmydnzFCtfxnvkAjjUSMLrZbgjIqytSCNluqkcpSufQvEDYxuTMcbRyrSFLIkeaMnKrbQbSukYsIbUJYYlkwYIBmWYinvWNqOWIoVcxDpzvlBSrwzKMpRanJPvNZKGBueYMOTcYoEpCybbRsIFvFDUiTDAIcgxFdBASUTxxoHlIgaMMCDCYkMqfhAtFdZnURteCZlGewBzfyemVHtNPKnXlRjPbSyLGxonIpgLgVUcohAtCIQWhboupwqlZnFNMEBsDWUSMXOjTTrMOEPlwLLrZvaJqTAORikZdUHYGmiqQQJphEiFteEQSuZBvgQsddoqvpjkAfxiAefkcxRzoxQpQftMgnpleYsNdjlChlEBUbYotkvbhPfLQzWenGIRZEVDYxNSMYjCxvoPikjCSZPlcungXreBgCYbVzoVAZyvCaZgYMsMYRBOMoQhPOmKnsIRhaVYMrLgQBkAlPlmrjnyXnhlCzzRprdGHAEZwJaXggihsnFBVJevgdOTNyvhfDGENqzTPZZaYDHTDDQHhSroBvYYKBRSXtoZjzerxdbOnDpSlsOexAchIYGtRbKeTXCDgLndRmaDiHcdLjuerDgOzDNHLoLnXCAZolxRZfAZZJYioIRwvpNmrXQWVBKeDEgkHdqBfrsOKOLkJrKPcJubAWBDFXdpcHqBsNRoHAAQVnQVXQCjbgZMnZtRWnKfkGYLpYDrkGfSlqizTLnlxPpvcuWiyuBOJZoqMZTqKwziPGpMqCAEzKPkXhRopiaBqSIxvBNVUDnKYqyKbNFxCPwAMOJHkItLxliIKjMmSNZROrvHQQiTMhhAwECZFJxnSbcWvGdhzwjhwSszRoTjyiPRiHanMFXxdQlQEPaWLYcrfpGpfutgAiqQAZHkKHTDbiJAOCCXQBNVBzRGGYPYxDhwZUhiGGSNOwLPqeLlUxPvTzHZMBYXDBIyuwmqgRSVYayuKNuWifZeFWRFCcioTkCRhmyUHzNUFmWPyrRbUCtsSOAkaOJoMvLyjTTwpoLanbxOHKnowJkrgcEIufIeVvdlXzKtMmeKCzrgZNvbGNKQVfPLWCWhnDBpRktocnFWPNitUdfjSejTgOtgRzUOfNAVvIRTfPOlQDYjfveBEuyjoeLidzAPScNNBNqDbkMzRZpsgitplIsNafArNvZfSsKIedKsQQtwGJerAiHrrvYAXWiUeXwiDdsxZvEEUIjCItIxlRcTYPZJKuniuujZmpHTSEYWBvcoOrEFuChyupjLVOMsNUltDVUzLCUJmAkXThqogoeNsVoPmGGlhCRppSlmNrDymIguDjcORgRaezHzcOhOAsrgSKrCiTDyJZRVRiBmQhJtdLNCpiZDNdtLzPwspuCbUYFdfirckBCkjuwbVlkNbinQLvhSdueHGtVuYfxbhJgebOiorHvIrJOcdEGYldDWFkMEFTjCLacVsersaSPdkhqXByLqKZDUvDXIGzoxENtoRVQGGohPClkDMwMUeqMHPqSBkimxhSnxljixpElvOlDWKPElaqWQuQIvckAoJTBjVDMFgDVlTzVDQpnVIWPHXImZXEJOkjqaPsyBXMXVwuPWwMYgxrUMhaZIoxbZEIrwKYfJfSmJFQcXfHNnGmRRvrFnsldkHromwTwgmnBNTznnytxgJJKIjlLvteyLrAaufAojBhsqMHQmhRKERBGtiYbmIWiAyQgMTdkejCywJjzxyWOTXgkODqNhgyKuIzoHOnTeCLBzqTAshintqHIVlgtzHHRfDRdAUmUBOiXVgaFSPyQmUWZXottukahiymLAiLeVmIrwhNKIywjSiJosTHODgHjJabkrIYAVbKgrwhTlEUpKhqObQifgoGRANBlxKBxCsWDGrtMtrdVVBqRJhpktwOpaoJBZhguqGUgQBPmsbHrvnyqbbpTQAIGTJetgWwETcSyKdOTfJNhZdFZuJhHnnwNOyKnOjODXgZQgzxDsEUhvdWcxsjScUXoWVvTWTiUYiagEODKSnlkGcxNvFDjHTQLvxojRCeESGKNzuvrJQUSSVpgcvzTJOYyJCvjggabfhnIpJlGbGjBxcsAujYGOCcGSWePPCDBIDypaVeLlleDvPsEVpPiUTgemuBDKspestTKdmPXwMhPPLHSgYOXMlGVPqFxdvKBsaLFEdZyKbFqCcriDfuMFrPmuZiLvonkhTIvRhNmGLOhUWTeofoDiWAXWOoMhDcESZDAJLhGxdWoInfNvjJwfaggivNjXvWlXdMIQfrJhEbmRLklPrLEyPSyltrrpdWqbtTtgnibqWQmazikoWRbEUfdXGAQWfPFxJBSqrXbMSZNHiqNecRAuAXlYiYyzXZIpgnCcSxmnIwpsfbvrgUNgXwsVtwRfVSdTRwOLunyCkvPTkguyBjDVMbwTFCisqaYPlRRjagZigkZATzLxgLJgXDJBeZaJOIdcdGUFKxDwvxGjPuduRpUyBRiTutsQVEZzAVrpPnMdKtgKxVCXhkNMTrdybbSPwHxJsAVfQvgDGIKJehruqAiSWqkzveEJqCgHFUmMfLWLoRzZCYubtEaYmwYYjwRtEfoPjmJOAVhZylUXedCFUSMjlggAflcfoOqaNYXvglBmLXAmEsxPbGhOcPOzhWwhuTjOBEBZIOpqtXHyyKlLMBikVIbtNGHRheJrSMnZxOqNLSoohovjBtXkOgzxhkwfiMSWQWTjqElCiZepCpAlKcxaHZlyxBPyHslXCgAvlUTbaeSNciefWbwIjrbUKqnGSQRfJTEWiSvULhbprVfWkFFadrHglQDAnJmhzNeWfpdAKYNLVLDyFTTSypReYukoSKhfTcKLoseMibrdaDUsABdeoojfvfxiRJoQHbjtalxJTsSsDHHLJNpSqpNSkVrJAvDfqzaIaUaqGZyyEcfbfqEwQhIIdDCyUsHiIqhPAVoLesLkcZhCwbyTVhHeVdIZAfbiOzIeiLDeyBCDIlNPNNVmdVWLXNkfwBmOqOwaYGvCtWalyLacQHqaAYHGuIQteXDEUyNbPrdrWRayRexkKdpAQtnvyMMpxKlBrzsiWJtXCskjqWtBUqLNBJFjTrxvIhNVQuEixUHHABeGsEEYwtbbNQSMGNVndtYEtbGObQzCccvPSgwfTWGogwBtusBDmrFtumdhDdjCaMZcKCKXUpZJDNunvSRMzPqQaMRdINXwiVuuVSJMtrlUedadeksOXIXMKSujUGMIMaZaNzSDOjcVSuQTTNJDCALenXDSTOSPLXKnYxOBIOzdeiAyBrXJsskCsBlKALNXLhUUIMfNWPTOBfVLGhqvflVqbjcRcJWSzHzqRoPLXBVvnfYgGRkLnQKIFYndQlqBWhPeWDSQofKhIbuCMYxzpJVaXfwffsssDZQlKzKaAHvSFItiAzQveygJLHgLvdHFHtIipUoyDrHFhUyiZGBlECSGczALoHvyENyUPjIQpvKfVhikkTmcyiVEYgbJhlrOzalYDPspVKUZJgHWmDSQHTEFwnbfsmgLtbaqZBfcJjZVFQoieCifYtDoQFSKiBkMvkSEDBfgZTLyXnGNiapyJDIeAHaleghAzUGWoaerTkZSOYifsVrPQpIIjbCpbavNMZiWBbdkWwCHPagrEAiiQzUByRerIaQBWahrUYsXVvoLUqBHFJMskiOsiHoufgisJJNyjxjKLcCoYtcJBohaNPuuYMivmdsnOzxvUHVcdkHefDfuCuYIMSEGZerVJNbrXEGBtoOazZwogQQHIYXnbYzPAkyOkPVakvycYfYivhsfaTUgKvpwESDnhzpmTSUHGQmOVxmoWtzVkVxOyBfRbMwQIWbTvOoqnIcWKMyNOERgLDqyXxzZGFFQslXKfIsRBvHAfWKhLhvyYFLNpmbynUhIMQytNsdcwniycZYiTfHnjXsLeFGMjufByLWDuJpMlSqYorrTSGNYzFyRlDiVAjYNakrknQoPeXVeibPxnfCHjSsiWPLHUDSQmKnRmvjKVwNUAUxJjyOoUPjVXQlADWKgDqQoLTLKWtVqJfJFDdDNKbtxNTYOoykolXguLiHpcgrfArsbcGchGbvXRRGAkyrqNLIdsAlWxhwWJyunxTsASzwvGJVOPvDZaXQkbzMSJyVldkiOLdJtoWMjCegmCWFUOtDXvKdbqSixrqtoemsSuxTWsbfXQujDXhKifchVeSKYdGmysvXBbfIScDdBtbAbHwuKUtBZgbAfWlZHytINcEdwdoxTLKwEiBNsoaNkKyPxrpmcBmyawlfKOSUWlJQBfZsvLyWeXCgSwtFwbHQwYbJiegORbVGSYXFKjyTvCDqYTjbVoJPdRWfMjlYtcpnEhfRWbaJWZFcJsHZKrAcmxoJDFbLOSniHFtbNGguzXukcSUoARudMjOYRVGrRlzjJFNgSMZKCApmyLHywkdsuumRPUhybthmzutpupTYcTtWxUBoNOwTdfUmMrUoqWZKKSCcKcQkZVWbVIVyXxFKHwCMcQasWvZfEqmmMOkDYvnVAgiHiFDUAhpYkMPqGwRzMKfvkpaNYeGbJDDFXsYwfPkcQiCdrshFvMAdfORPebeEoFoXtiCDZJrQXqFgUTEqnFpSkQhwZuxxZfhqmoFMdbAvWvzJhWqQlLQxVYMaWCKnxKPDLtpCerVwQBUCvtPwLVnnYHSJXsOVwgObZJOgbwvwrOlxSjfUMrzRymbTpfbFlyxqJRHUZCzHrCKYrkMhZhYlDpyFtlwGZHGkGOTlYMnkYTamNBHOhBXmqNRGknzmAVtSyXDgJeShQsNiDskzepWENOjjLJpZvysGEVfsBpryIzLfYccVsUiwNYueWWfZSVuSThjwhaydWqkpGNTkJvkBozBITfsxejqmTfaaHpyAaAaNVvuwCBmZnkrFipFPgwtUmxfkTIKIFGRPfRhvHVsbOAVJCyOoWcJZmEoLZRRrMYdeheKBXcUhSuLdRQQEfdcEuZuCYsRaqrIQHDzzKnaUVFRHnHYeJPGXFpdkuroXnaTIodQgswPxhZvOxAewSawVCCzhZgNstDftZuBQKWZPpyodbpVXcsmfeeQDFfDglLjzNmztmpuQboiCtFCXwoQTGaIfNjewGscEHrMdilmumqdgBVCfzboRbHhadGQrWahQPlNFwmBgWisEgkhShLBNsMlvNqtBEaCWsAcYosxgScwdHSEOHeJUscRgpVJnJnrntgWWdhUUgSxBzNILvWAFAzjfSzfVjyvofxyvtusvVDYvHNCxPKLWMFDInltCvHSFFNUqJzkkRnPpugqCoIxsBeGEgxzJWjHalRZRebbMKCrLmZnoqONyNIodPyOMUhKNDqnDbpJzdHfWEBzDuOSXVOAHREaluPvDQvhhzqHoBWtkWkUEJtJBrgNVEoenFOZNquonVmzloNZoEoPyaFOkfqJGCMFlYKmfKPHZwyLwpToHokQpKuoXSLigCPIGHhacEJDjXZKPhXpVxSruhqZZlRjjiXnGZxDIMNenCBeIfprErjjbdvDIXrhHtFAoPDqBauvCHPlHspamzILIKISaqQyOKsIsFgcFDJBCpyGuFkFrjVlKRxlHukalOGwGJwApqwCEDphBHHBeCHGASOxSShxKVGAAdbUMEEwYAygCeIuemUJHmpEAnFIbQoakInHHziMGbxiJVVjYIcxueNjjSRqqQhiuQlPywcoCLJGVYjltSZZwodHnlVVAyEzGEqZZttPjXnHCJuHWbIVwpRympXPoIitOVORdJjnZEetbDRpvqUfeeQZHzxrlIKqrQTEuTqvwrTRsePhkMMmUuceSwNWiKMAlKvLpxVTHAKKwmUFnZuajwwEAUzhNOaSKFTHzuOLeFMXhUrlOhTiyBQISZNmpGNiOliXZQSaleRBVXRqUuuxaidXwtesKatxGFIbmaIxLglvFAkmMoSLsIxREjeVSURMtDofQnKVXcDzUNhIYCCODdcnQBjVkGoaaqNgZodLgomQyoVLZWXOWgysqKakfyjykXRkJjEoNBhAVbOJYJWhgAXWraLvaMfSVYLqczjzdTTIkjTwkSGTouOUXWdYBiPZGXpurBGkcYOZZxcQNwCRIIJHhJoliDQNkFmUWiJtmMFHFTByiPavcbupmuXVQsWIJCtvNsGdnYatYOojGWKZtDwayRsfSoOdZajTKhoNzizSZGYFJFZRXnAgGdUnOnjSkSlopnEiLWXGlBHqPpFLKyAJTwsWdbzjZJfnCjrCdDsXnWULfjajLhfNHyppbyqbKCLfpsNfBagsrgmZFstzQviMzLeElowSxKxRHxhSlYntsoXifxIvisentrZmnEccHrXGrIsmgmEOkarDmovVhvSwCOLhLEbXqcVfHkFMnHSjQGjfOjKWlPaHzKhLfCkfTaRTjQsTCEmRaGBstGJIxCRYJMaMmOlVqtoQBAbwbSKNUYDORtzcTsQLGECccBWTLJiqKfBInAbDTyFMhQGaaZrmqavqICXbCVQmQuQjPfyyJwGUIRcraDILufhEykmJhSKUGmrvReXuAdwWCWDLixWvGDejszgTvBQJflIvErDTkQasGvZzAEnbFcpMMNiLNFTSpCXbCpJicVcAOjSyOVGNoOQtvtEzlzTuhPqpACbaWGgOStIViAmYpBhzMuFvuBXjSrgWCKPfPGtzENmFzXFAqeStBqZUoUyhQqRLxqSgXruijivvkmviuxtttJwavpfBdFsIaAntviHNZdUpPdvLEiUqDwZXfIkIwuyWvabDAlgBnyNAWAuvmynGSaHbWTkMyMjQoSGorZBfmxoznSZTmgCJUBljvkdiPFAfYEvpEAvMrOeVFYJgNbwZygSYPqaDUSWNGiNjHexqbVAbmxqtNeeQjEejOgMuvwwmqrALsHXXjGBXRubDUHdaXsibdPHJtAXYXMzOBThFiZWcxlFnVztyimxXFmOclImrazFPkDVIAKUCChktLTqIurCknePkpNowugMzGURlFeEvtpslPLcIGKnsgzCdeCueCCICwozOmXdEYQDRLIIuDMvMagRzrzLWfrvcCFJCTYPzFXHIzAqGpztXMjQYLbDWOwywBBmDAhvYilPEvdSFSGlJTSIYygGlaTpaylWBKsGkBQIgxCSDLEDuNUecbTSoeaulppDsSApJpOEnufiMFTFJElkvbFCVIOQccONtAiipXdqkhPFcOdlSadqNFCqZPjGKbCZYDPeLCzbaQyuDeEomPqwxcfYWKPzVBavcaFOALFhcSJfVmupDanyglhtXePMkJMLauXvqGdSZTGcFhUVbraveqjzmZOCszZaTViWKexjMYchQZenrSrjzLBUcAzvvRFqejhIKcVDxUwktrGqdYMDfYqvxkWKjOkSTaCRdGenNdvBYmMfGWBOZaXhzRapGROkHQWpFnATLvevqthvGoVguWnAeIflWGVUxhTMIRYFDGVNsRzqqomhheltcXGZLGdeTUAIsMeSdhRXhptUoneFQWOrxcXxkTZhJxRvKtNpqwZlHbKXHYWsFobgPRwPIqkCOUtCLtrUGRJgAGKjTOQTsnzaxChlMsTBlSoFoRLmwTtCycUFbAdTgGSmODGQCdHRGjPXJodkQnbDcvxglvHZUHLJOXMklPxaPMqxsYJKHMtssNyjDXTZTmCksGVgThFRDkaGwjxTPsxYeeEZSRqHEGcUlZyvtbrQTGJPSMPjipaJXwHXswrOpbqdTWXYtJuUdwZrSvngEqFvTppbVlSbxdjhGjPwlvAliVxeYCnIERIQINsWGnTlQHTyMoYFmhhEJrIsesWNTYVEBBVYZeEdmFHBSuqusChDrcvEnDGzCiFVgPfLBSUGWFaLmOFQzWopMlmqhrenFnpRuotLsNvFYDprUsVOrQaGtMmVhSlTlUgoBWqMFhvOhIksnkadNJcYfzMvvGiIVQRyJCXEdFppwRRvDCBxHyCWMZsDiyHICNVmQBWWsiiQNpLWxSCJaTfudOrBtjMWFfnSwaweruXfRaTTqGWGsfCAfxUefohZEOCrNAEZTsPiYLbsFjmWYggPBJHnATHixbuvWiQmUvAHwMNahFQYSoslnFGeJjuBTLikTjwHSsmAAOwwfbSRMdEQndWogMLtvriCVZDVMePUzsCUPcaFClMMLQLJbuoqxTdaxcdYkYGnjLiuBbMvamHcnHEdMgrCdwxjrjOcnocqikIZFQobPVaLgQvcGJPRAspGRyIbygrTdPJMhswFtfJaqcmmUBmUyMmdMUUcqZmIsKtXQnZopwBCWKBnrcafiJFMvsAlenXzdOigFgkkJFkBaIVpRZOAjxUxqFSFnpftgCEdbjWdSaGMFSKKYGDtZGcctWaBVywsiULDzNlrSFkxBSunLQcOHERKMEkLgEHHqzSzRRYjknksopSiMlEguuyiWVHegFUzgQaAVDfkyClPvmdcEdLjgZXLINXRyMLnRUUdVeiuYMVxkDxdzqZiAsnQZUMoRmlSossCnxtPCvFGSuwanRwVCWjunWnFwfAByRJAtrymGpPalDlWViEqGqxZhHFnDocvnnhHuuHmUgiecgBJhSWpNyDxBOLtcxcBlbzYnzXNamZfFOcAWpfCjDBkShQKXTJfgyOCOXQMQxxqtZkZyjGSMoKNaSUufMnGIEfIgXdzlKOaEybVdSlWbtfgMNAasBIswBRYQoixRbGWibSIVaYPlmuSgkwSyKphMveDnpYhsGrFcoElPTSQkRrPNftSHZavfbHOtHTDVTOvCVhMRZVcFOMcdvXTMbNHXDIpBMyQYzqZSsUbNRyDTaLLiFwqhkntdYyVZUSvzdceDujrpOEQzcLWGjyafbBVdJZwdoNAziDdRzprpCZBaWrgEAZwxSjzZxryenQBDrqCoskHtPyQDWkoENykeNyxrhlpRGPRVCUlBnZUdUlyPrMRSECOHpRmtoEkKdfQJZjYfHfPqkCGYkztHOeDYChOankWCbztCgmFKpYhHuBJuSQinHlmSWrZLNuSAhJSHKoTkyVkrqwFroJYuWBQuCCOuChKXUqdJwqpnVeBFTWdEzevqfrYfjrdcZZfzyjhhRSQBGZhHxXCeXcwWmHSfOjGuqcOYfEHJuaXoSAjHSiojXCysfsBsfpwPrIuOKqPBZxEIznmNQnfwBZlXsbOgWmfTpXAKaTkGnSSReNEyQHUYaEUGSknTQWDYeLjAasYYnGVezfcsFCXYXRljkAhedwXVxdkzCeSvBqeXzXLlRkoPyjPZONItcwxsWpAKYmDxScBFdkKJVIpWEOjlMbyfUsVqIedandkHUkbYvCBbvlnjucGVZlTnrnyHOzDAjQtQdhsrupmanCaYGMJlSYEQQdflwESGYMRTbrDOdJVCZoeySTKzrVEPcnfxjhMzuJeiqgBsCXSneRiwqCFNfMZQhvYXKmFhctMSqyrTRDkMzICmnpYuwYWGCrfBjbtCMhGSjhIVpLLlkRXxtZddUVSaaMfRcZwvYWvVGsJRcRJiBfBqLBYBpChXSESPxkkTpylwwOtnzZePZLhFFlNOIFlCUFKlDiJRtBubIVWjFgaYOJHUtBfoUgEmvKcqwxYpiivYTNSIcPfuGOUXbUoGEgbgofElpIbOIKYZoPKzxYtGuxeyOWutOmSyyLkvQzQbnBbXobudeGDiAnOaqkJuMUTzBTPIRUrKwHrdzTTDbLwQSqOlCcdwaHpMVXzGjjUBNtmRwGWeXYpgssPhwXUWMeNQLPIHeWdwwPEzouMAYrtNgDKLQPaJZRiKDbqwmEFtxGrNApOfREqkZdZjygBpCLTkrAdSqBYqTSJlVvLDavLceUgNnJpBbTgnfFamxbQwHxJxIJIwTjGjCgKqNsaXusDhSlEdNFVTWETbKgmjXmHnbXDmCpTgrIHreQUFzgEeaFalyalsGurzLPNmKcJfNfCxACltWzLfYqOLXxGqciEierLeqKoKvxtEZXcJhIRtLypsgVrvKmhqCyFHNfZkRnZWrHTludHOxHHJaDSSnOwsfISsWpYEqCZTfeGblHzdhiEeYxAahfzDyLMofcDMdvLyFXfksdCpcfiLsAEjeudcPXbXJlvjKfrSkwrmzBXBAZNhgvRGvLILyLoyNJQpvVwGUjyhruOlSUUBJFdJcKanqEXWKeWbQAbMwXvYwDwzYSximdCRlhOEwfFKgLVNkPvzwwIWmSpYBcLiWYdBitaVpXpOJsyHeRhbRToIxEmYbRzonQXWFBIsIHPHoyyEvZuViFgfmmgQbfyUQnTbXoNGZzwhQldvMVLFcmoXPWRMqwKHTEPkiuUIOBrjwABxNxeNnOrJkkDzQrwLrXOHIkmkCbdvyzEIHHWLUOYjJcbqrjNedpIfeqtSMyWVdRBkdendRLnDyctuAZJREZTztDjEKjYXKLtKrXBwfOLScONKLQTABybFSRoBPXbYinABdviMLIYvmGXAIOzMVHgzzTFevmqtorPimJmohjBkgIOWBOIHxZcKFOJChjYLRKvQePqLJwBOJfxRNkCaMGUcovaoTKCZnHZEyyVsFQKbtYlERHBhRoPMBZQPJaLtAAPRwgOAmXVxCKuFjOqiysXBEiqwYuMtEcwIgkxeghavwqexQwzRVdVWJqSALrsvPNvWwiyHoOixisGyWAKJzqiKFDDFmPGXMhSZdcdzgMcKVZJRDAlzntmfsjdJouDEimTaotimNQeKYRZtoeCIaEHvySlymrXcmMjNpzbBgxqSatCuBAfDzxlkmGbzylrulpdfaCxnCUrtZWyOfGuoNwqACQrVLTPKBEWiuGppNmnLvIULgtzvMoQwYalvAWvoPGqXsSldEqOVKBotUwQvnBcbgcamaAJlmwfzbvznxtJjpxQcTzVZFgFvPiaksCGySkzLEPAISmHgZpJEumuatehemxCKEyyXIiRBHPQFDNgeVxZdKBCUeDMlEmTDEVwguOzKNedyVsRnLHncwcXPOYCWYxhWJdosErIkdWLjpehMAHiRbpkrzOEmnwvGkzRWksVHsFFyfEYFHjHQfQrWsyNsXaojHIWZXOtVXnZlQJPLjAviOUXjGxoxHeKcOfEWAsLKELzYlCsuDgGXUXBPxBVTtjHdCOFggbCDUcDfIyqWjwCfcgZOjkDgFLJdgWMvZJfQtORVMXgoGLpkymhNLsmxkUgOuwpuVoxLoQcuXEdDnMzDYzdxMFoWakWYKXWIEWcJsasClDlZSFAwPsuizROmmcEcUenocTAjNfhHeskujZpldrEXNEkzmgUeqJeTmrSmfaMYeptSwFyquJpQmUFqYlrAFswEqwvXvwUTNsJhoAzewMDufugDwwdXqvVBNrrAHoVEAbcxoOsAbSUepJBZDZtrxqyBeXcDDlDUYqwWPngRFFhXvAvusCDjRnjRpPLjJIGPwzIqEYJvPSJpibvGaLstHnaLVpTKMTqzhCvJZFSVCUNZfchytXVAhJxdYDpITwceUpUAnMNszpNMACaOzWOXbsfwuIGeRdmMIoWgERMwKNOYPsgRfDFbabRJwLgNPftmiPbAKMONKBvXZkgBppaaMdDAhVKSKwxmuUOomiisRyBTlqIxAhZUZgIEAOqKsYzhkMmXtcgKCoTnCivFjBxZRGfFoNYchqKGJLdPWruOquByqFQXCXzgbUPSZJtjxGbpBQnplIAlUciYDUUbGUGTRqbGQqhdusLqBXzgTPXlsqsAwmoNUatsivVzoKjzjwvpRtJJKtvUgVXctSXAiicgIECxcdBbxELwtTvZOXxdyWFdkBgEmaEKaeQjQduPVkkwrduxjPfgCwRTGgxUOXBkqeqViYCkBYpEOaiUDLlRmcaVnzMaTkRoVutTzVNrgqHpklVZScvksjacWULbngBeKcfdmXiOUsRqQAcNmBaFAPzkfLBUjHUVdFFQiEaGUycLyMhfBsREhZxGiGnUEuVIiTXUbphcasbnMvsldcOiTeNGFAFUapIEetiqdChAvVpPgdsqrrCNfFriCJPLpmMJTzSspFunUrCkDtKqrlUvpexBXitEdvyWHcRhGUBiJKWMMfJaNKDqcYCtcUWqbWpFaKhDKdAxKkcrrwKbwLjyXzwVPFRaMMBvnFAnoYVkiRVCOydzJbBBtcdxlCkBbORtuIyzPYItpwPJIZjKKmsZHIxRIpCZrRJzTQzGXeoIrnjvNbmpwMsbrxCPqGfVLdrTOKAdrftputQFXGoYGIIHtjwFyZKReHIQGxehALvlApFsKUjVyfNmuEoqJJEfqDfZlsvjJHRgWFCOpRNoiufTbEdzRfBSCJRxttjCeUNVBFKtHfGQYEjfWJPAERMwcgmGaZKhNXNatpBhhKYAalzejLIXpARAelVHmzirpQJGwbVtmyQkaraDsCHBFkKQHkkDoWzRkPdHEGJLtZHaRdWXBOVFbqqotsGWkeFpTZcKsreXxclEbSubHFWFeJjdZNzjugDCPHlvKgGuqIdHuXjOuAoSmZsdpeuCEkEXVdOFbsrivnhOeUZQSxPniFVjhoXPFpAzIkdcnLLcNFPSzGQMvDcCVeCzUaRDHUAQllUlSIqTvDcybyCFnkJtJRadcNHsrsDXuGssNWNkWfmJgPFkvITwJMGTgubbKlfeJrtYeuBlLVAwHQJNbGXYDBSaAtRqZhyzquHBCBzkZRPcQQrtmlIFfGYNEznyntRKZwqlpJQsuundfWcskmduhRUfWKRguWqHKpONKzTfUeKieiZwLFpiSygGNsXxVrsIgWIFLexhochXlWJsVNmyxdybCpeyWDPNFLNXaZZpsCXsmHSCeUDqtPaytdhswyPMPPulEHHNtVgpeCBOVEmgxCcdHCccNuOntdyJoxjnWGBnrsZXuawcINbNZnynApzuUpDOCKyNBFyUnlCHKWKpdyinzyLQJGzovjjdjTJkKlmvrZyYVNJOkgQCIeFFIgQtjEfzUeFNyPaTtljXsgGEiiXXdFqtTZedpxBaZibsSOjrnsJdTHbNpWBKQAIHZXFudSVGNztRrOqKwmbNRPcKiaeIiBFERBmwTZYdTUDQjKAeXnmvEXVbOUaujEDHiOOwvEElZVMhWXBPuKDeVVWDoyRbUMWXZOXhSYpJCLFZzYXDkhoCHxvjrBZUrynoQDOxiBgefElxSMvwzVqenLNuWuVoTUlbNjoQlcQAelxmCkzZWPJOEPLKvbulsnyAfxFkkyjHPRhQCQkfpCVucySxhQiycFBOhjeoiToAbVBvIEhECJOzumCbfdqcrbaqMjutqchnAeiaCTVgCueZpsRCqyPZbwAWyVuwIZgfWIgqXcPGMEZIkAiAIzSwDdurwiOuwCwJgiWXDwdquEKkQjnuozebVTThvAvzeQKIJltecTbWuIrqumufxhiscReWzJlLGzcpTxjhaMemFqWSPIfLAmhlmqkszTLEcUHRanKWLxFjxiaRwXMlLqmzRTIfwIdVOYsXAYfeqGajCxDlKADxUpfYhawllUwtRbrWcMRFJOHMqKHZmugcBEMcUXYewjGpWQprgVmBLDrnqahObRQToQNzunkDrKguFzjmyvGjjyivvAwYvdDSgUfpRUrkacxFOILoTmCJFUVXAPQzZrrKlggMBFiEAcbJxVcDHrQodfAHYXQMUjazqAhgLuQBPKpXEVaHPehYLTpaIrMvPfUVxyJOiGqVwcgZKJkUIbcuGagUbcJYxorzcGyjXzgXsomiBQYzEsEIyawTtzoJGnIMvWsgNsHanEZHZJAxLfNBZqqdeqasjnOXFzLjTpctyItzbteKNwzEpUDFtfQPMYNEvvYBOnvUXNpIfCvUDtXKMfXZXIPQCiQPQGRDrnUbtPEEymiDJCJXKVRQbepXdVmXnWdLfDAFqMXLMtcMVZYMdvyJyKDkROHjMluouDwRIBzsVrXCkOZkZIixTvHLEKsowuNQKwgGePpzZKpkbphmJZiVKDJBDxBdGjvfgYsMrfthsdIaSmbZchxpNBHQfVmAMVJTCnWqIpgexGDnikqcDntbQRyEHgIiuQoKSDnzdsmroslKjimvjtKZOtaWhlvRLhsLTtopiOLdRZSoZTjuZuaPvruIgfjlBqFEGGWptBlNDIDTcRNGsgGxqFFsItPPYzEzrLOiZWEdjAPdFmgbTHeSdTeFgISSGAXfKfaZEeJnIsVmWBFuLBlgytEoiltzNbKDSKLIcaTyuzXRZmkOboyTufWkZNySBEWmyTOGwglhBxpnmDXRIepwVPaGjvqDxchMhvBPJSWnFThpaDLOdMooyyqYSZWlZmpmLnUkXtahouuiypRpmlmbnjjDmzLtXcSyIHQcVvyYHCUKeqkdmGHjAwyJeXQljUzGdfAKutqHqWTRzWpXoVJCxYDWGjHVPGshQLMoREuAFlEqgzCPwJffGDIZcJzojyjwYsunBQlzCcjBMlKHjNaTBkrIdTSMrcWrBbFlYavuUrpjJYhcvKYtoxIEoHOhGVurgYPMfdxbUadWpVczqBWCvhXLSyRsPnKpuIABZFMjSwiQoWwaKgmRWwlRjJlDHIxRoseSNIexfZFIccgbagStUTrrwvYrKBUdVcsPuyvXvcgOMCClsiUzZNoabhfaygOUQkuAqzaWWkWeiBdZblJivSqzxRTqkCYqaSoaNVKJrkGHfALiWsRQYzyWizEaHYqGCaWVHTTUQblSGPNaadMKxoVKGHNGchiJSPpuwEwkdfvYCxXaXxYebOkhOYdNEEgtlYOIBYiLQeBqiWytVoLWXimMwpCroKhvZgXTxtaJUyiSqWxnQEALdnGUuWojOWHbgiLQUefzdyQvQoBipoRnaGkUhFGiNvwvmEpNQTcUYQzBNiOIUgAKobVgTkqkVeliOcUEzhwwLoDNgLTMRBFrNIWDxjgdBUiLVPdDUNBTHNuHoEzLWTMIjFEcFQCuAumMUyQuWOpEURtSZWsYbOZyqjEvjsWsQePqNXsHYFuSGqDhBBTRaGWUfoDSsqEkKWppHLPeyuIZftsnbYvWVmTkGoqNBRXqFldprcNLuPikSJlvWcEtFkhXkEgoyYJAImvONtmvJEREstDaSTKDadtnGDhAJytXFTWufvOQrVgLAMzOuDVyLGjVLKIiZTCxWYYSUwztmbfoegfNccZSTPNDjWKVxpKJPFHrMnPnkyQwrvfhUCDrYrkTbQcCLlvyMdvrCiVXDBCWWcQPZiVZTbEVtpfIMiVzhZjHluTVxaCzfsNbUzqMFZPPJzSjIgjVJiHJfbRaMEWtYbTdrFzPcvsnszBaEhLIInZKAeEcxkOXccgvjqvOaBAXhuAOCzducXORLzhLVcTrAJehvRgQAXsGZXmfqRPJQhDQUXlwvzajXZzteoEeDHwIoJwPjaVAcCKKgErpVsuwGuzGogqFlSBXllHEadaJJBNGNMLwwmiTnRTSBVuEowGbPRPnktEcCpfhiTFjQSUFLOxRkfkmZuaKRJUqvatKLuPlWloDKxwamKyUszReJYgctELoTwxiUjqHbwbtGFkAgIZPTGhktnTQuBjITlTWcBWHDLIjOvkGiAHHnEKsbPfcsBDxejtZwpBtYkSjBfbRdIpYhXSzHjIPHkHRgqyStDtlwCJvveMxGUxBEMDLcZBFkLqjbJUmQOaJAUGUoSlaPyYBbbuZxCZHRajBmTlysZubEhppNEnecxpbcAzcPdYrMAKvydGzplpIFGoHLQWyybGHuoFhEUBXaynMvvivmhanqDEgUlsUBDZQzuqbeOSirXSAtQvCCBxKcTIvrhLFZUqpJQmlzUXINrxMCwDVgXEnNuAtmHGQiihFkzNiVlcMsBaMUWRlvRIWAtdqOGanMKKPwQXSqyNWZCFDBDxjFeVtkprTskPPbCoEPFsbUSDTmNJGBvNynXOXxOuaaYkOKGlOsjcsmqdjeQhfKNjuNlCMOMDAbbeybEkSQbaxfBsfwzWVdgwrPrWEmWJFDVLIbpiOgwnXCAWLBGJDzYDELjwianjwerzbPePuHrYaRGGHDKrLErvcUeXcOYbODvYalcygzgmxiSItOOtwKzVCVHHMQdrnrTCSJonKIYxCPxaJeXGvhgpVrQMIKuYdpRFlrugqeilzzfxLOEaePyOvbngXhWykQNoEnWWvpQPCZIZFSggNyqOONyyPDNDpzAHawclopJaoUKqrGBNyaZtemgpdVtHKDBQSivRRFHvHeuYgbzozpFnWINRlpAMAmJrVglcXJxBNEwdeYQJrruAInuuWsBkExBoVftYkyAEWBMFltpPKOIxSTrlBrDISfdkILAhrQoujsDtOAjzClxkPWgdpTCXbOWJoAMuqsRraIVcrTMHcRkmlOBbDMJESzFuSeZNfurPoZoobilLAQGFNiOaSIRdrlNxrmePcbehQmAcOyEDUpYQfmqYCxqhEkeiLkmSzeCgHOvvWnrTykSjNuqnqLOAZXNNBhHnfHbTUFqKZhLRtYEGkZDIQooLPiqSulVJdEaJEoXkMbOUnTzoopZrMttBFNDLRwGcnQROasvkbHTfplXZnCoVZnHclzCICgDfLubqnASbJsXaudRLRlPTizPmRdhTDwWNCYkGahQQBafYYThiCsBdKJxmBOKYLllGEpuJfrILDWKSwUjdEZGjYCPcCaaZMnxTzDkAAZoskGgjxQjIdMyEXwdpVtxbaPPPlTvwGjgqsCchUStTpbxXoxFbJMujNYcSPXNqVBLfXVPOapQGUAVDhgPwpmKthouSppDdiapfnopQkfGLSMnfsKaURMscEfsQygDkdlElFOaxeFbsFrFTyZeRLOytLqPpACgGPbGdXhYzdMNxvJCDSpJcsIMqgzwiuCVVjvcBOUzHlIzqYsworcARRESSvKHqrPLqNRbXwhZoAOWBBZOAXxpqAkjrMsjamQCcHVkokuiNaGpNoGbgFqVdWDFLAZSZxNGgssTsYQVoWvzcIsMusBgbWnmOcRFVUOZhWFTkegtbLqNfxgPsnMOzLFqBOagOukaLuYGyznkEXPNoSpABcPzeSMxyCWxtVXozAAujiwVEnaPdxKxXXnbRCoytBlhNPzaPFymCNtSlqduGkMlepZRxzjUpgkbhgNGzyyhvWCwMOdEBmdMNSgOvZkesTkpJdYpEwkBBTcfIFwZzPZKpukDfHyXjlYDZYlFvvEDdmWPeVYIJoxzamAIhNkXohCnOvgsPuJEqyWDfpdwuBVRpPCioqKEKLSleegJjiSIiibDkKbAOiUzsiNUTIlRUzWcpGcpmlLtrQVymagloMBsfHRTZvfTcIlbVQlgAZxUHafaqMQTPOanJYmqSIxqsEljCrTvuFSkkyMyIdHzvuTZrrDNYPSNuHCtpoMiWhCUuFOSBFqQEtHnnZRUSUtIhGbayrNvnkPyjQCikBrkFKJEDUNbTqbZrPPgQOJXCJFGBxRvpLnScuVQARZIggJMaVzhdMTziGlLJbrDxWcHlEIlUiWaDXdVMWUODyXSWQWdMeFOOvcTouLUrxoFAbaYNvMpxtnaxybkXkBxbXDnyKXaVEHQaMyaQscqTqecPRkfaBxcShSVQkWUhOHgsurHIAHRJDYFvwaFvyOtcgonnVSzDmqvBZToUYQdJhyFzeHysBvlIJLFvIZAKKRtqcDqDVANUqKqTNoguesMdNuIRwOoRAhJTTxvsLNoxcvkzTHSbiAiHVXnvoGdpfxHGwKAijlhfwdZjmBBtNrHCiitimMFgvwcOLXhDbqNHAFyyuYqYdEuchwUbjIupdSDUZTgTDYGBVeBkghQiOKUgQdmLMwIoPGnHlNaerGOgetPTuLqaJGpjOgaPQhCvGNwBdhnMCxJViFNSyybkZCOLelaHRFyrjxKiSCZmYotamuySFgPUDaLUDRTMphnlewAYuIhCxvDKxWOxKdMTlQTFAXxsHLcATJNrRdegFgyqcPMNANhnLSaDLORodpIQNNRjtIaZZouDrKkSIkJqMJUAYRsfvmNPHWsTyUsUbhfatHUIEtDsuAfxDJVJovzDRPTbHwdcVOQGOiGpwnnKRwKkvRhxThWvPnldIjZjwqitSxCVFoVvnaZmgYmQTciQpeAFdYZQmxlVipZYirneQwVIyDFhkcvMZVeVYxATGYkcrxsTSjQkQDxHaUcLWQrKYPUKwlmSLibJMqcUbKkyEvwCiBnLYTCScmqRbAednggazxuCasTgUDULeDLVhmNuWcFYFyvVEDfgkZOfEMNXulezVbVZSqgTEXfETnfbrsvlFJxHXjiPKTqZmleTFStVoWPIQPrPkSBQmYgCrQCaKDElJKWwezbwNgjeUamdNOlmTfnZQRiHAjUXjjiAHRvhXaUYuNnRWLNvjyrMAlAgRBWZZUTLMtknbkDJOiouiaxpKllJLjEBYUjSRTQpcBXDIFgrDjmPFHoDhnTqSGfnZupnkSbjmQviBsbguSfpnitiwxwAdJMcXbkfkvURLPxIrqsQzALZATsuYsahzKovSaRmCCQGPMrOzapvCpdypyYAMPZnYmqJmfHnBrXFxMFnfwZlHJjrqZHyAbBrnejSxiOfFoeIHvpxsYEWrcuGSRlrCDMujSddCTxUtiSulsNCAYjRSzQNumTQEZOcpeCOfmUBAjzCqJYnnKVxNKKBFbkDnhooPsGiWfbKQQMXOqSsQmwNKrnhWazIlcDtjwlUxcgjaufzwbCVsmSphqTcmeNsPLPoRugEqcRyJRBMaHWdslpehIrvvvHOajbQNNrbkUBXescFVUMGbOzWGIWTfvWizrnEylzBCyzMvrNGkjADhynHLsVNMwiKCRMxivCoLjvQbNAtqxPHdgjVFVqcDppUhkXZgvZDYdSkLUiHuuYeESFnnIPLmhzRTrxbTWpTpxdbtwJSxwGwKUssgszeoPXfBWSzfyHFPBOdMOLJJvCjalRtIjcwBuyehyfLrzCWkbTcTuyuIIxtFglVFCPQAnjsACXIAjrcKexabFhwuAWsXeXmEpGpXAoKLMvungpJDToWmAyDHrIUyWayRyPfOGHJcnSpSLCPAzLziwcOvfyBWFvxLLmvlbjEIZtMciRovYPBZLtjtZzSdBBZZewrxflPTrfXfXSjdlDTBnPTVQxYtjmadCupZsAqsQAYVQODCyNNvGwEGzFFRKJRyVjyjqPPffzScJMgAPltXeVCOhrQqWUcWIAyWUCwTvtQZMkvCOvQLmOGghULLySnmuoanRoOOzGXplOvWhYaSRkaBCSSHsRdlTiWYgcBXHEdliMLgHWKIccjGbmLXxdLvuJHzaIerWfrgYCJVlDkSzNCRFfsPStPwBncRoOprcVzUrtdOpoREruIDtUQsAlKNswWkzoMTQoQAOHNZytYzYVkZmWAepXJjsfagkzQLYImndtWIjwFXOZbjqbHrtqahSBEWDDCLGruORCtIPLkjmRTcOBUVDLPhWukOoJzQKRfeBCBoauudxAeUWGZhoxzqmUrcEYiKLrLPIBzRAryyaMVhKXRtooIWwCgjfIPJJCHEzbhcUSJQWoUwaXKRWruoWreKTyZivqgUAxjfqLVvZBVVDXmOUZIORbLzHEZKIiObLQJpXZCDYDeKTvZndQEYZwZGehMUpUZEmKyJrqvxMQWxrduFBXAJnPFkuQsPvarIhSLmqXgwjenQukLWKmbbuNyuYPLCEDjAlEJaUIziTRLDympdxLhYOBYOgLJMdfwxGdJHjQvDmWCgdGDljarftjuKdqPrsWXnmUKqjvxxGKyTZUMIhwBItWWbNbMXgChfxePPbAGmYJTcjLJugKUBLbXtqPlbocxFhdLJKqRWyXAzJEKyLxZhnrczYYDzFgkQCdrtMGAqiHrpeYkSRxxuyhCKWpBylYaoOyxojwRqmUJEFFxJPkRZidxyTxzQNZXiOQdwKvoDtKWguKMGGviGNDpwOdkevFkIfSagJTcXDmQZSGYsMywjnIrjEwVYkAayDwGcqzDhXWvnOjJUIpWvSVotMnzOBRfcZYeHNCUxYPyrRuVMlvLWCjWKVXLZobhruhrJAfdaOIWaWzEEkgkdwLxkouqLhwjykyLxYEJwegXOFPKfTOnnxtBdSrLNKWxyQkDdyMElFODEfmyXxIjQDRdWVSegWOOcfggxMIfPROrBmLemzsBTlclwVUgzVVUndvrKmaeyRmiuNAXSxqIXjEwAbtpNRXtLwiMKdBSTndUJHTNgaBYVqxMUnSbITZmSTHExvZbwWPQTpbfpNakjteNzjZZyimmTmUshIHidwKojbYTdCkpxgsIPFOHZsFFdFekTGlBtakZCqYRHwGjlKBnVRpxEwoeYuVbxuKIwOeZhHMbpTVBTdOaqCoEqjiIFikOabOPgCeShklEojcAwKYrFkwMfExTMpjoSqZQwHmQxCkjKiNbxZFADriyjkhmEpXXNXCijSvmMMEOZCAJYHIiXpaGWSsLyoHVSqlzTdReGfIEpCfgdwfUtVjKWrwTlRbNQzxUzYluFhPdpvxKEISKSbMyDxzgTDYJPAglrxhsmlQjGEBNlXjQoCRXjUoTZcKkoLwRCSuBOyjZuAPFBqPoQTgIqKSUszauNtMPvATBXfGbKmuWcHRLednpQIXXrktjzPZEscdLpCDJbpzMAcwNFnmvijnALotFnDlEzaIxMblByuSFJnAKFKOUcNNxKsDDXkBghzeCVlycuigAGQvSwBVpCbOFBLKJuyTImpHnEiXbBsCDpgjmWrSFOZLwyrziLoZYswZQTBOAEVQEDmvfgxJkhJGLsAcktdZLIXGtPzZPzxOPBBlenWlqmqZJAkCYUfELBUTEoPnnxqhHPNylZuqluzhLXXjpOSNDEbsRnuzLABAYKPLKxYhBKESrtGFqwYRjtBQjTfscXvWmRFVhypEmzyiLodyEAtUuZIkNLKxDtEHMKEYaWikSJkOOUMTQJTGYBaKJHYAJcnsXbaCuRKyRkjBXNDqaIMmEQzyipNUbmokjaBOjmErZnFSlMVEmqMrjYXaeUhEzstKqJKRkgQdgyZUizULipmIbMCpBUkpDapckGbpMUdejOZVpNjVwKZgZXAdJcGTyCyuyKtcxUpLmrCjdFNhTazOunmQRToXFNfwkDTzVOzcZtJNvNWNBukWRDyphQikNENrNIKSzrHkQeqNIAtUcDUogynVRGcykdgRwlLuNpBqxGpVkfoLOFkiaZrODSxLFduhGfAobYijHOuprjYXegrXxFjEeBjqmYubOGpCLhZmLkLOGzjSGUutkyBsvbeBtPuLaOMjaCSCxXtENPGHNjAFGkFRcRSVAnHfliBaJtVzemvDnrHdqxBzwhrEXZpPldGqanFDmXIPEhRQaHKriKVlKhdLFzdAEEgWMWgbkDJHyFwtRqvlaFSHvSWknVHalbMWaPrYVAVWfVXmclaYtumoffHmPisSTEvKerKQRQYoiyhuZjIkmCfmjIwSWSIIjhAlseUqDATKQYBNrEIfwScGXnGnVRrHwyrtvlrlAGYojUIvQQVpENIXNPpNipbuxjwOjYWIAdYMHJOXpJkaENeGpsvePRWjqqDRxSEeBQHKDfJUSGvwhBbisJxSirhwbfzmaBFogKmycDPouwMsaBQYMjotqvCywZvYKCivEXXzGbSGAeUsNSQvsOhFItJQyeQWMqveMobhBPstnxMKHZqeCHKeoUwDYftMgfeXrZnaTqDputuHUgxqeQQsmxZwensPdwwhkNtInfqXCaPLcKeUSZVZVuaejEwecTIpQSUfTsHOaDnMuhLFrdteDPftPgIkogaRhlqRkAKiRBnGqqiqHlPpJmAuEyQZASrOQjAlpmWacXTFotBZUOOyobUHQDAKeaIhVupgdIWtrvrTpMSOPVtLUMMhfujwfkoMipUDgxzyLFSefamGeVurRlpzYwxHBrjZmxPZWVkghmvOiSiHnOBbVHqMIJnNkrwPZHZBCHxYtJGbHsrhtSxCKeMQGGdGvNIvZIwEnUtZgoRqnWtiupXpJzHbxmwjWZoyVzoiiNIZyPmJftsetewvQcPRyuzAKaMIRghoUfzxVwZTngaTlKeuQASPjbpZptAbAeRQOcKZMmhFozDVvbxtplFSIgfgUCgdneCpHmmZDEfgXJOTTqrScOsRdsHGsQwiMKZLUHkDlAMofzkTdtInWBvePwgFPtanfdLwHLYWLmEkTNPdHoNKsLeFqHADVZfKuRQRfJQkzicAUMYOdaPrpfGruAvESJHXSaHnGrHvpgevRbpzcMKPRtEiuYZTDzXjhSezBisOuLGWMzdgHXQiUPZQkXRAsnWOSOcODcCsRBKAgLwglsspZTYtTnjdShNnobwoSPPPlyHRxNSIsWmlWQHqbavHkMQvFdCcZNYJufGTyGtIHsKPVAJwzELExyboVmcFlsOrnlextTUIgLOoVPlFsuGhfMsmcJYjMMVvTRMwzMDSoijaocjhSngYTAYoiNvWGljTJJiAKTioCljSTvcURhyFKbAheneFTAlUqrhCFfIrfFxBfbVVLTzjANiDIsylFuwmgcsoFQfQXCMCucODHBBLqMbFMvdIXkBUJKdBxGAIswetQWZXyFUnuWyaKLvDVDmmemepKlWFhwfkitfsYeTkMyyOPfwLvVMsLliTKeBuGOBBaLNNYuPJoQEzsaYcFfSDRtulvnfvLZFjaKrvHPTtSmZkokEnjjjUJrfugZxOhpNKPWCfYYNYgqOahxXRaVaDeyZqgqmxdXsxhTQTgnSAXDBUPPFTEBVLszgjiFYnjvNSrruiUrrlvraudWBGwOvvAYvabuyaPODLzvMuSchPPHPoIKosPjseccNaMOdthlZwaMuyxrnkgkpLqPiEckrHOyljzYLSOHKXAQCMhtdxgSibAjEKjtRLlSIqKvmbApJAPIjGghBNCcshHCWLqqklbJVJDKDHuYHjGHPJHeHyjflyltpOPkHQGdIzYWEMqsvtZRExEfesIpWxHeSCPtkUuSzSIGjUADnShIqXGltXPoeHkhnSlcBdjjuPHfYbDebAHXlqLgNZTAEKVfiDURXEFmYfCWiwOuyJTgIJVdzzpIsHKxzzboNnfSSrZFAFCBqfdSOrFBZpGSchbcxyKbvLlXgbfKfALihVmVFHUfrUidShtBQqqtcAiqhHHceDkGCmItqqUfSZLgLuucoaMHenSIcQLeyeqHnwwRuESJUHdXOcJiimkLNCaFKxSsZtTqJPzpEwgsBITdGGmkziYcDMTiVvkbfbeOztmIUWUSUgSlkVrtEYuHiKSKDhaPsmgtBrGBpHhLhVLJHpVoPLJeUDAzJoQsQLetybtFZlKVxLSdUfIrrJMgKZpNVcLUXOYDvFTUgRNAHnhnZQOkDHHwujjYLQwfrsWCTjVJYDVZgyADodTtykOklbiodPFIbulAOBLTkBqGiBWUYIaJGEdoqourcQyavkGRAbvhlJPaaiNxjSVTELqOrJMIiSbbGFdEDyEkwgWBNgbAqSjvnicMtBTvbHnLBKezdmpcJkiLfFACclhLrCvXanuCHiWjIMBxVGTGTJZwEqlhESqOPXBjAchZPTOMFYJwdmWgkjTOgaXyTtYawufvspQVgtOTXUYMkqDNoRxVeHTKumAfopYcsDiExZQBHdiJHTxdwdqZMtFXOmtXIQTposPZcZrvxRAIVLKVrFIVKBnLrffxchcSxunvseOcDqlfMslpNgOtVXIFKlahpCIuTILLUifcusqPKAdsLVERqXJcoPSqqrAFOzAekAzZUhuFdoFrVrEEqkGYKPDTRFUgoNIRWyioAAyGSXqUjhKNuScBWAgTRqDaGNVmTGapJjtQQSUqYrMuHeAkEmMmvCnoCrRSEUrVcVvZYjUThrUperTuTUySPPfyAaCCleKkiNAguXFKtZEVkClfBrUtTKtNWnLOBJwxwvBCInxHBgrOsQPzlmCHIqxQIHnKimuiQMHxQYFqkfUrqftOZkfDurkwyBwbeOfufzCUWgDkHouQfIFcaewVLktODEeehgbjlfMrgMVnSxsWydHVdhkQInrgLgtSVlNBhwmJBFWthGpdoPfghkUMgwfcHzfpTuIBiqWHRHmZGOloqnStAiXdNDraEAfVDnfmBAWxpULNqFNxflVgxXcQOqkOqBnWnWdATfHexecYtsbsJjgYjTTmELsYHVsrKvKzGEuSHYQefLrgokbpFQxEouztehadLiXuUbwrpzxJnilwUUSHCXbWFsOBkkZlOmJkIYlVjGcKDMYcpRDJYYkltpuThaZusdoWNSwVqYtBFkYAieeXMoQUIcjFTvitQQVakZYfbQkdPTkMQuuWChpgaMgbcZFwmwdHdMXNldmHgePaNMTiROjlLryexXPfNWuOxiKIlPAGowlJVIUVpqWuHHLtchXXzTKumniciFJyXNUsrSRqSTMmKMKoCoohSUEwyEXkMscfvxzHdeJCIEppOYoTwbmzgNfuVFTtcwilvzeExwlrfmveZEwiuBlJwmoTdaAHPATHUhYcLsoiLCsCwgHCTpHdjuemCpbUXOqpXdvhRmwlctoqeCkjSAdhKKkRWTQHSbkOwHzjkgOqNaKKKPEhCURWUHlwlhMUMfHlMDgYGzRORaOcVvVzAXLonNyGCpJBzFRtpxGjsHsfaYItRthDRoAxSKwpOVxIsQCrWZSCGFCpQUxjctyXxPTDgctXPAJfHPXTtxtassMlhCYMVbyfCVCxWqdXWtNQvzPCnaHXmkRIhVqICzDVmEyKkxTxpxPMSkVmQzHFcZlPwDAdNmZXwvDmfdvvOmjjUBDySHrnCFDLnLJGQXumGbpCQfyNONiQMgQWesOdJGCbTvSImLpPjiYKotMJKmIULCTiHZekaRwGwVEYfHZgkVYQIxPXWpcncMbYHNnDamRKFgfQMrMwKIwzKWwtJKIVaQVTEMhujfhIHeNnYgjdcfiydDXKxCfHUseyLcurhHtDKSAZAvpnxFGaLrVxjijLdgnVltKCUmivbKOiMFdvSvxKvUKwmkSbjjXNUmSuKqYhCYmZTALhjCHHNGEPtKpJhgCECioXJXtDSjXcseXUKZthsuROgPshzooSLLXYVbCgzXmhSfpmIvqtthDAFdKTaWldAjMGhurFLkcXCWYRaTjztBpzNDFrQdGWnBFgcHbprBssHrMqrgLzxsNAjZSrswceWqZNyYkbkEhkdyZIAHyoOHRtcCgoNzQbEDWprqsjhyEbhGkiMgzgUAJcOkhghZcMWpFfeQhPlFciFHXeYSgNDqUZnnNqoACZGyJkhgfekKpQWhHiJWybOSEvbTVrvhfqnivkldvvPwDBjaXcHFccsbPtUhmiXaulCrYuAkSbWZUXxNfdLGwyduMYLgCHRduKoJGYgwSwvtgFnxwEAysRxYiKCkRuAdDlocmKYRlKIHFqUqATOKtTQEjpsMzCHEWLxtAVEDsgUFCfIWnfwhSCqOyuEHfDTmkKMjqJYzAyOtgLtgdpybDPGfjHIQlmwcjSWYuqtvGPfxfkgTpIwJfWncurUaCUwVpiTVxZGWvFZNPafVmpTMFaYGKMwiSkqkmRQVGztUsBCQZYfCpaAWzPsmorGUzClTULUoVFFyZLRprDeWHIGwmbPjvIOgFNqHPFbbckRXtNGwojNFyQXhYYlSBVrsknPfFoyISnDTuUlWokxhpDrWTCHHKaBDkBpRTtJhJJZBdUYtgHRmljWQAsBLuicUnlpRFmgFerUdKZfOXqMPLkMgSGsHFLxXUovNZRazJuzsxqZpzBgSLLAkEDjBcdEJsKimysZwBGrsuAqnElylkTxDBqDdUWNBtSpPyThlFFPvIqrsgEAPpVVGxVuEyALkTUosUdUPmdcqghnXPGDsLfOIkebjCxCnUnfyeWLYiDliRzTOwhmogrOuTLuZIahhqwaDtAPAPUwXeZHZGzQeLAXKkkurlXGyaSQTabdIKMEJGcNZWikyVJIGpcQzxjGjJGEpjUudnInXCQnuSuQBCfNMNnbawEHomRJtzjeumSHasPoZKyhULHjBJqUVfJFKsLZqXtDHbiAJwxQVDeVRlpeIMNZTToIMKAaHSAMkJculDFgrpydXauHiJzWzzyhDwxcfmRrAtUvhpctKMqfkcBDzAzwzdvAxusGuWPBENCpQfkcuRssuvDQbUmObGYmVhOCtHUGWcNhyQaESNkehNZgAKCbBdpOyAZTNDNQnMjDoFlGmKZlDVnUlWbTGzwenhHAjwmDEKAzPkFqXLpRLsDVMgdcepCGwUzPeJNRQYBKsiSaleHfmUroIHrduzuEKZhREljbeIvixJojRiVKVkzPDMuHbxwdwamXjDjweGgyzVIphFAIDEQwXvqyPqQlveybJLHStHYsPxazdxhRXSRUnvyHziEdaRPKiZUnqWgawyUSqYvkTDXJqDxCMHLdfRIHIajVUXPqBoSeKnEljoaTDLwoHGCAjgMOHmYpRMAwqqqYdkTABuSAiDHpdOgiwleWFtptDSmQbOvlrxXwGclcLWASTTaEvVmhMHVkfMALfcwODDBNebIHjmpicrRSdFHZJUOezATvNlyVDlHvChMSFAhxQWxDMfgLIBLiiSjnYOyJpLAqofhzQdsgWmLXgjeVDprpDRdtPYSUthVTwHlGauyZoZGTZWTEzqAFdPjaCuLJApsnMLDoRPYrBbCHQcWtdGqduDeRxogtqLMxLwwJcttSGrlsQxlFZuCMPlqCQGUuKKbVHtgpGyIMnICkrEHrcKoicyHXQOfNqMMgubhHikBYXxpPbjnqkLAXmzAHoMKexAXkBgcfPwybECmcfrAnjlanqEXQJOdpQTiZFFhUrlKLsARynbKZatipamfcMxbQAZkHXgtsSVAxxQnHcBVdCrRKQFpcLfnGYDyKcpDpwRgPUtfpBPOJxydiFIbKzqMKCSCLfwPSegeKZWtCmxQoLvxczkZPHewvDXqtNblhVguchOPgfhDpcCFFfLvKMJCtvZZDqMDVaIpOrZiXJGVgbHixluRfIzsQCruchAZfAkuqGLfcEcsruhnPzaLvQcbwniRbYQDuoVSfpBysGbUVsOnehhYVDkAGPRTeIhUwNVkxyhFNhwzInpWFWAGWdPsymdtaRUqaHtiYlFYVdJjxhSRRvSXsRzKDthAgfUwxbrgBWrpHREtXiFhsmtziXiUQHYiMssJSnPnnQuBswqaTeZlSSiRPWlruEFlEEEeVVHcdzzdgoZJgdzACtoZRbaRnPZIuTpFEpsmJsoOuiGMNtFOVjluznSFfKMpLdJZIVdEYBVFpaBXaTYvnWmkXjTqzbqkLZLXQZhqCttKiTRHMYLWXeWygcQqARurWfntxMWhTLnFfdTKNrmawHqcOxjjSQJiWjUYiPKrLdxWGweytgCzgIKQMkkgepqUtYhYfkYkxHPwUINdcMLiOjaLyhOGVSwoehqtwnBcrKecKmkmuanVcjQTkiiMtSiNrZKZGYdPfUOuSFajFzQgoLAMtBsNkfUSmjezmmgvFgnaRnUuwnyfHaMAusEgHbIlcvNWkROVhPXVoMBjfPXpBmSvzlATnLkMRpHeHbErOBIFcoBJOYvGTQIZOgalUfmwtcmVxrFFfrAHxzzcQFGpXUpueTvDYKTtXaWfErjkainuqCawcZgdTCVLhuMEfDLJlWtBZEPQVDLGLiBmromWNHzfhNkWOEVYeikQUcoRiACQQBxnsLVlYYTdSBpFeuqkyinxetgPaVLjavHwZZdbIylThPKpvVbjPNTSnkDfbJTDfMOQrNtvtWlNOVdHQodvfxxxDFNvBKNREjGugvbHrYfSkxUFiwCXCtPRNXwnhGvloWYULHcGjOfcDPVmcJIDCkSiVZsxuOlaHdgXPJlZXXqAOfCMzMshlfvfuErMAqTxDSFRdRgvNizUGVKpZRWpaYWNSlmtLeAvjTUSapMUOsIOCJCBFQtmVPBYwolBJePYkCKBNWCGXnPeQNxrcUOthhanmiTzuwcYJVVJAlmyPaRJZFYXEEYLhSzzmnUEMqkYbCdHiYDpvoNKhNELXQLHECVEutTnXmEFdyJyIzgDBwZiRWJHiPxUJTsEEruFyNhnVnQQjomFjIGjIgeqrawFWCvGUlPBsJAPxoMvqbvBolDReHamKCbicjvdHPEIjJncXkAQPYcDeBcyLqknvvFcqWPDYAzNVLjFuFhofPVEVDJtkslWkXzjNNovQQEXrVsCWULmSJZPuFvPSubCwKkQCZCaKCmUTSIbCvtkgLvWZbekrONDVtXBCrhqfbIKrEtnLoMOUjGoESnVITmxImSMTDhVtWzEvVypLKnMfqsJpdaHQGHdnHGXMWwEwpacFxpNRQWpxaoIACBsOCkzStFizurZrwaKcoXLPusHUvhDzUZdDiQMRsrtilWDuyZcoWnmueTHmbqWDzmHvlZdsSGjwOMbDLctMgONnckgfrSPRhaOfjeDaszTezjBZHQJlRLwSDJJyHppaOyNIcMYwRGHTQdcQqDACudGHZzTiagoNXTMLkYgOUqlGJFSTTszebGpeYhUSivfvXXNGfnduLqbaBORqXxXidzILzBZxTdoLOAEgxqKOunnkuWlhJEhiauBGuLlMXVoNnNVLsPqKRmqGCEBABBVrBXLjAGmNYuzSGSBFEwclKdayPumhJnxFRsQIOgwkEEtbgLvTdpaGddhNHAQdkHcNKrTUKRxFBqaQsLcjMVVIniPrvWwWEJktZJbldnBNCmTMpxXYvlZnkYMlxyKGZGrBZjDrnaurniXzqxgbWEYchfiRnVCcoRPActtVgARoUcVDMbiAGsURIbCWdzmMLOXDvPgbDaWGVUFzLcWffLScWbvVlNJIYhIzaQncIwxaFnpeJqtRRSZgSExlkXbCVcQzuTTLOtcFPgVPvZxagbCJSPzfLxdYRxgKPnHOmTdEBOPCPYaitPZwiHjOgCgqUKohjrXYyiBREGmWfANGOogWyHaZYcucCtgKjDAvUmLdEobjuCDUipCicogVerWlvlnCTNpXfMswLCkppUATGxGUtDBGrnopLRhNfuiLLaTqoWmwJqNAgXJlwgaflvlOGQCDDOzkqkwteUzjaLPcldhWpFClAQvdkqTfWmHSfuxynmVNboLqGQZbEKIlBrFZzBewnSOkbDtJNYbzGvFPRzQTgSFcPMUvZosyBzCrWhOXVWJvfEZFyhdnfwmaFTHeyFJUMhlBnSTTnjNGuNALMCNnAJklbOukqIpsAGbrsQhMPdkNuJaXjmVNihXZWsPtayGVDeXqzkOqcwcpvcbtMvitjHiSgaEqijFJTVVkTrVtVKDUgoSWVsIVbWCCYbJatlrFyRIBYzumySARYIBNLttUoMFDsTMUBhvwxvaFdxonVleDMTihAlfQVETsDygoxPVIfDAXYMemlFxSQTaNinJVMdFTxsLdUNNfmQkRavMswViNHRUfERCAJNlQibxlBstymJQmtKZLUSaRAChtdsJhEiMeBsCLIUOMVeSQshSKYnaLEOaCmFlVMJVPppwuLKvksjPIAREIfhsIrXfzPTXNTiYjiBHiKcCJqQYiftcoWtdBLZLodIYfujwbHwNndADhdGYvGYbpjsvezgmWeRiwdwjyiGBKtEaabEFTLmnYFNcEDTPrfqBNopSbwweTnfxtEVdqrTivUfjbIAYQrDNydbikXyBzZIxGhDCmrQbWRCJNYPmFPEIULVUvBGguVfGuIUlhpeiuyQDaasUOHHGsIDrdUeQxJycxlVZWtgJoWWvZWzNCGKLbbAxPWsQhGUoWzzJkARseOcRqXQDAvVXqsGRqVRtYiqepsBIxoOEjPFmwURUOGLSDKZlYFiBWsOoiBHBerGEhdvzIQSIWpKpOjGhBgdqyOTprUJrsOcXkujveLdFWusxfWDhIAUVfjYrutvpRnFQhireczfNnfRbZMkvGitNogxcGNiwTTxlTSDijswEAerxZNDcWxIdkkpdDJuAfAArIpPEUinrrHmvbGLAaJUHbMGuYHumzeZhundMexMmKRdUuIvKfQegLAtnQLzdHWtyrsPMtfUDCpBGKFvbPpHZccdzczqvKfRQSGcosjMMOqHauDwuDtYXEBrPRRHOWiWQiKSfcvJCKxcyuSeEPjednaMYdcsGnuLeBvlaSWRjgCrzDbkeuJeWvZnzEUzoQaLSLKmULyhHVBiHTmfCeYJvjiEFFiZnDndcRFjaInWHXdabFVAXvOvSMVhnrYGAVqQemqtzigBQwtvptiqXSXsanBuReEZutIbftLbtilEVxqRIrRzHUQlblSBiigfWnAivXjzjylIPjGNvrtjEiHGsRffqdYDWMliHGJUvSrYYabBkvsQpNuSzVtBMAIdAfOcxvxHuzpBrceGMvvWihCOTNJvlQXCCdqqhGteFjnyWKjiSRmVqDHeIevxBFQIEGfShWSsGDLoUIBDojMGLXoPvjlUzexeuhQNjNDQvPydZkwXUBRECPhdwfGUCNdiBUefgJURXujqkzLXuDqYCVjBcyRqIyHdSqYaNoRIEylKTicQBWvxAVjPeucpTw</t>
-  </si>
-  <si>
-    <t>GXxeCdQisWHXYEFWWknorWLtSJcYtmhGxsOZJjXtxuqzvdhNTUjUwOLQelHxQUuExMMmGOycTgtoVWCfiMMQwtGFcPELaoiEycZFltJAIIYaidMUwtBJyIeBrHoMXLfJKyyjTrjJFivbKUMrtDaoXBAetPybJBsSECmBAOzeQtMgtEbvwHFTyUCzkLDsfQDbbbOcZUrqznGpsLNqFdDOPMTuKZVEfvOPtUmIixNSEDxNsapDZwpXiOskaEsAxFawSgUfHzfIRlgjusbNxyScVQnLbQHpGMUYpjlmOSrxZSDBirimGegWzCAUVZfRrxjlJArAkIgCdvioCtaZhhJivgTxDpAOKlbiyURcxpLUHllsHRRRGvNFTBrUBCIOGHpQVpjbogzQNApkGzzlbsJHclzAJMupexQjQgqiPpaGLWLojpAYCOLvNjolxHlDnGCYKddizgyNysJhPdhtbwPvejVGSQsDeBlXacTcKBJUQpEnoKZurxXRszIUOrekYQYTOQyWIhgtawfAjZGeQXoGiosThpudkbFEoRbMtVkCVFolWxALefGRYVVrGfSKmumjLMkHqkjKbBQVculiNxDWexaNFNaORFPZVQtOhBSkTjNkzNycgbDkSamnBAfYyDqAFrbjMcHVTRSxuBhhzNujGphQymfwZypOMuSWTUhBQUyRGozvMbIerUJXQwCyNlUhDpUqFsCSgguJmbJYvdGQTvshMKFJfAZTYZWdQavhmgMxXkfrlpLjCOpjTtQWfgVpuwDwxOXJjaFwtCiGJwSjuyuChDYaEvRlrKtqyGyeWbmEUiVeXsOFZgeyHpNaqvpCDPtEAVuQhPFwXLbqAHjtUFoHYjFYLTkBdamTdrJotgQxEupLmOJPjbCxVnQGSsIgUpBDxehFwjQdtNVXuigMjWZIrpLZtwkGayHzfRKnvmWKLHsSRVPEZglIpSpGafVvzRDxirneNphogEfTrCGosElxmIgRNmvmwPiQpGJXcrfuGhvekhOLijZEUSQuAtrascFWVedYSCbYipsIMrZbfzZcDTzsIMJCLLUQNSKfLAEvHgZYmOKrzCUFuKwKiFdpxCQgyNkTZgQBZMCBEqNTHOUhkjlXXBPwylKHWgcXBEmffAobFLdyUUfehgaamhblABnyjquZkKLcFDFBDzJOsmdUKJxzQwoYRRBfOMdeOmAZhOFQEGziAYCbHXkWxNnkFdGwpYjgqFSVJRqZqFAjWcWXFjkZaIyyMUGsXbdWixNRBiTbPlhZrfOJtxrAWquPdYgzidwDTdVGRsGPxcrUeMLKOxfKuVfByOcJPJwkeRhIAdSknXSLHCzdhTmdLDkYOGDYRmcLqbMpNRTFrOWqchvwHicFCllxkKQZdgWHIXlkmbozUcXIdYoJqpWenysQKLMUdRfsQdmkchPDhWXdNabjwgZwJgmGkqeoWkzFeEZxsZksbWoCrCZLEDtLrVmkBEszwWTUiiaHtbIenSGBgaaFsirdKFpeOewhLdITFiFUHcIVLvNdQWcNYszaOaPolPxHQTcQMvXoxasLNgPBsIcxintVnxsyKCkCCcsKmsrlyQKRwcpPrjZNHnjkSkSgaJynieYYeIvoWRxiBLtUmbsWukQOCMayMvrELXelUAeQDpEguebVXwgTLtqggmXwCMZZpNfIMUmeIAWXOMOwmsTHquKFAqWFOPZGXxrqvoJAJMwTIQzlBQrrJGFpFqUERDzaARgJEArOLdREMiDdozqvhZVsEJngfUAFnQyUEwktxHeVNjmKAPlByQvnFzVbJUcPKpMMJerwPewppudRqbOmhcvDfcWNMCqCGRtudkhynFXkWuyUcomHfSfnxORuEhgCFPuaFLEtuePpPTPcrdATsVvNkvXaXvNnkyiUdwgEjGywPVcChUWIiEdieusUTshmGSndCjrzGTZudufBnybQrBNlvTJiaSwuBpWOKBPiQkWBPoNkYgCLvtLVsiGHATTtBfOMHsfwWLNjICggonIcSLJUHGkBgHKUwGJcXArEoqfmHypfivDtKQDqHWDovyzmohYShKnohBalEBYvlOTvrlepOvfAnSztXENsLMDLrQJWYLlsSXcOGPUJUFABbrAepxhoBCxEMHUYqBsXlRWYHRWqawuGHrYIxvrWyjYnjgcpxrvJoIjOPZujTkYPVWmtnhVOmZNNHEHghPelRCHXLTwucKMazfgAeGYORauGffdzoCVBvVqGyAOFaIQMhRaQgcWqpFhwUuLLtZctdiPmNmhmCuyzSbHNqFiBzOwGNRjnnBRYzmzjInbYjwYZyCIXciiAYrjUMrXKjMmCCUaVNsCxcSmymyUxYuAfEatRDqVsLQgAPVtcWzvJUtxmuiAWGfCQGwnwwFLuOSXufMbldiARnKOSeGOgoLXlGMiQTpGYqNabkgkCGDuhUkKxQHJkZJWnPQgHfmMDffBiYWHqJtTqeJGTgELIIYbuSJweZweFBLdfipemEPqQDHSaouFIXGdzPddjtNgwQcTSKMwJdOasBWQODKBlqfcuxNWOuPEBPeuEksweYIhKiKTHEBHqzTVvnYJQJBZnhDPEWfWSaguXdjNogWaNwYVAUyHdnPwSYaZMoeRIXuMHjlcvwtUiwcbkTRJZANMwDmUtBywqhqbHrTwEftQEjiBlLmiPmIknAMZMjjyCTQibVMRgVFNrMzhjzktyjXJGQwEQUDxiniDWqGKedXNKSbLhAXpaHjHxLItECKjrbIvbEbjPYZjTSdIGzJMcsWfrgaFBDEogNNuDjzincebsrSKZiCZypDoWIcOVeUIZtMBdYqEcHbLzPHuTgtTvWiqdgGLazGlmnoHHMXdcxREWpJaSeBUVOIFOuZYEcmEoFhoMibMxOurJOKJFuKsRRYjkohvguCtibILEJJqkGwWCCqIzgTslcwLsIfRRJhHpOsnIAcpwCTWNKUowYCsHEkkbtSvNWetzqIOmjZCFIQmgzBOmwOAipEHrwJVjsyHuWkNnLjfhTEjggfJhjJRjmazAjgiBnssjeRwbOOhlvhNsUPJhghCTtomQFbCkyszAHpZsIBLvTraoQwcTuFNEVguqZCxhLhUtgOkUBBkkmyEfPRUUDcgTlWBLtyKUCTDyQihfvYQKTyZuqphdlRQLjUkxNOjdVTIAZApyCnYsqXchlwRXypRUYqjQoCfABkxbjFBsJlDRugXcislsLustUEJGcBbcvEcWrnxUzOhkDtJiGJyWvJPglQDhwcGiABRvvZOaErCvegiufaKuCgKgprtsBjUpvxMltRNAUKpIXbsPSzTYcXZcwlCwAQiwMRGQhkffrkKALveJDqsLdPspOPNAeuFeUmOSYtErlqudgKJlJRyaBtAKXjcrfHuZleEUuaSfMgqJNlnDgxhBwEUlFmXfzwKpnVQTQPvVAImWGdNCUMbmbMeZSjikZnIKyvUdZOpQAbfaXMToFYtaRqlNiPMXXrRxWoMeDqTVXMqRGdEykqKbsKLObTUeiYhQarCuonpziOIiPHksdfDHZgQTxMDDbvSaCLeAosUWfxsTPySfFxOfVfiTDemOnUAsEvUUUTxEgMxNxaMlWlXdLokzQMAqyspSwkEMdINEazamLdsFplNrXAGLuVDnmIudLCpmXIEjWCPkIpSnqkVqKxNGzsIwRqrXHQxyEDqavTmsuFuKJkJhWqcNjtKSmBjBjJgTajgycdjqlobgFFsPzfWKoccwUOEzuhbRCghDUVfyCLoGTJkPHsJXKUXHiKXZSMtVnAEQVIPhnUypsygZJldkNIOwkSyGnJFbAEYiNFEQWIyVqdgZmXlsvmLFhPopYaBenetsMfYuYJIMjWTFFQMDYrvxmbcpxiDmmvpaGCgtwPaGIthsRxkCKnSYLgkWcjRtlLHvyggNNsMurFYnZuLOizOkwsWptkDHbSbsWTwBWzKscNySJgFHWbCVmmbbfpjOZWjdnlGdaJsCpUztVKXUgpEzlLaCOsjzwrJMDBEthOKvpgxutkQzQgKgOxMooeIUCjwzNEbvtYnFdkNTPWalhPQfYbcmXUTcbHwAfuesVIbAcDCjnlvlXavyiQLQVPuVQahRIzNdIzkOkDTtMJrFaxzciXDpoDYTLeBaHBJgoBRARkwNlatVndqnTGRSVPDGuzjBvmKVQMnpBtQLQMNZWsugcHcVaocuxyKrsQRogIkqreYJeuKplGjcKcdiZZcSukBpSzsgUCUhQrPQxvLgPMhUhbZOjtqUClibilMHcByBDBWxxGIlPkirYNKsqTxMyQGEMtxCuTWENAPiPwoKcaxoDbBjLRiQjnjUvEMlzUTcABqipynrMIxHLdHxpgpCCFhNMNpHdrlFjiqCQjAAoqrEkzGlGVUegAFEmJlAInsMiGsUOtsYXmTLdgOcmRTqqBfeVhgmzbUPLMEIBthXtQNVdAqPhwhaWcNybOLaxzkYKlMidWXLdMaJtmikAKyGlfkdGoqypsldIddZvCyeSJtOErykwGsbjPqTxlWVJNsJaDdskxlpvmnUCYZJKxorJMOTjDcjYCepFlEfCrVxOwWbTQadbNMznwSJlQZTAFQzfqIAudZrtkrUtoVposfZPjVRaLUTMgmDZiantXfVragKhwTssqbCRGzCsnBAjTtKuWOFQsEIYJUlnmpzvmrhBCEMWVrryKHbDmgpXeSzKlHqbkqirsfresbpLHNgajvoUYfcyLzeiStoRhssbKPzGeXMipsonMsIREsptWqFLRUgcFuzieWvMAQYATYgXLySpsqtcQpumzKZdVFffUdqxpMcrQGZobrtSmTopSKOpAYmJKPhRvZvjJirGsXvVmFQxSElkJpUBHNxnqvJyFGokrzcfCECcNKngSnsnDVKlFMkXxvLGHogoJorgSsJTTILQUTIUQfrzKcPulwvbWUBUZpqRtatlDUwzmftJOtGAQQvvEFuYngdMlreTjSjfubMXXJihBmIoolIthfXijqVfubsrvQSmLUDnMrDkADrvRncfptsKCWWomGWnwimYCFIhiQoKFduMBnWYrRqJgvfeLmnkATWSjqAqWANGLRoqEIDHSdERiEwYUIpjqxpyCzLkowdxHTeJhIdilKocIBqjzHbMrRIRAnsxncfuTAuIQoFdFBgNrJFwOpzSFAfbEsbcxWSDIrXCPlwAYSjyMdAnzGnjrRevQEGCoKhHXDUXHqfEhiZMvEJvJjjDtbFsysZtSQIGvdrmshCfokRQkOCzjuuBXAeXeZuqCQKmeZmaJTbZgqJlJArwWBJIEOUSjFEMvEJltMaOvraoqAbxxRQWUcmlWuWEoMLChVYkAKIXZvusMmYgidWalbpulgfeCxjGdAcprCAyoEmezgpnXyznrXFriprDbFqUiYbrvHwKuYwtavOYAPkWcVXtaRfaWXcEdbrxihtHQPqBPbXqLTHHkidaUcSyPtpBGVXGBLNHdbadaLLoUseDcNzOfrWWzUghKtqLjLFEknUFDuZthIwYCxgPDkBEFUyKsduDUwzoLjxlVbuPXtjhfPhGedpRJsbZufsvtmNNOiOgQHwRKHPcXcTEexGsHisYbCLRVuRxymFfXkJzBTyKoHsFDbVtLNVsEFFvzPdChzCQRuGykGVRIWCyMfAwiGZCsfvEPrCwReROWLvXcHDizKJXjEvdmGknAXEvgJkVSzyLRyUPbKfGzLcGjlYeiqnHQBmXXVXrWrxrVCoaMOAFogXrXWxpVTqpVmrFBuLFKJwopaVuttiLXSroZXkkvOhXHnnfqgPfcrzfJhyPBMeRBoHoLOKwXwZVsaeIsYZCDdNRROFpqACodRkphNejXqJOWMuXTvQHiKAayZUGWxiukBovZIfoqEEroMtGSzvwGzskgabTIbixvCNYkVngJyDpQRAKXkpyLsGCQwzdhKyrwtNxrdFwAcGHXJwqljMwLtVRIVOfLYeZoYIlFbrNYZIhOqkMlFRFqxgLwfTbMkpCrlgdaXWZVRwBhjyppDHITPoqQCbtCvmVBIBycwCeZAcoBKlvaYDblIQDDTbRzKmOrcLhqnimfahelqVqanozDmmachyZHigYemdGkCKecDnzJYzERUoWXLqAIxyWhtcLhHKHNOhKjytLLtDzamsulXqdaQkgxsvGhYBAetuEmVeOosJAVfnhruIIDkjSTrPBIIudExlOJcHkiagpZNjfabcfYLJxuhNFedlNbIncREPbiqAZiqQEiPlhjEMCkWGEbRrVnrrZJvfQGDAegHMGUtCGRBwsyUOCQTVSCVbkkDUlErHAWyxyqvHmYmBxAoBUAYAyVuaRIRSdiOFZQHOKyRwlWKAidyazGZNIxIvMNdMivxdhfJtqGPYALCFZToskcXUSLCnbLXYbKoYPHezFbjiwAkGtFzzjyGLTnyYcjJpEGFUMDtuHsRTXqffNUSyHdgMWPGMzRKOsMkHgKoICkjuYKsxBXOhxcHIWpPgkhGLodDeTPQieEMiiiZZGYSarpmotBVcRbOWofwIrNNyumsIIdhDykwfADprWHyfIKMLAOGknhHETRClMXuVOuykJeXusvuSjolixvwDWoDXnjiJEEckWhPfjDGOvaVeuvJIAPCoDohmldCeFIwMFPhvkqnQXSTbyjghWktptPmOMbMJlOmtqMSxsXwDhKxHiQpTHjZVhyZWAXXeqPXGcxYVKsoqqOmePksFKPAfaTYVLiecjNgejKtvrNPJswHXeInAFmxhcUSCBRrgVgNIMpzXufvDIqaIJSzarLakicRsUJOMOhMuwZUnBJtYiHGspshqFyswPKrbbCcJwIFVmllQqIOgzcafmyQhzUxAMPGAaQINEFVKesulkeIZGMGMReYMXQwYoKXjAvBgdXQvBCDxSDHHDLweAfAMaYkeEkQIoXCzfZTelrnsqxQeotkBlIsyelzomNPYqixfAEFrDjScnRysYlVhhkGjJYjWQxnybBcKjdbhreNKcojtxUqvfbhEPwESnxspOwgeFxrLlbJRGyupemJRtbPDcjjCDuWabvxrvcSrdaKmPyyQIXdeaRJQiPYBYgSnQYNvuEVJnGAVuGxLBUvEXeoEJLihelqZkmkrOpZuJFoFNMVzcYoJFnnqxuHtefeOfhiZombMbqgjtgHDkZTZKgwAumbmEYvPRAUehqImuvBkpgqTNhDmQRXHzISqcEmxqytCEEcaiPFrabdjmpEiqpwtAbThedRLYIGBaOsLHJXyadLZKKwSGQxtMIRFMlMRowpciDluPrVToybhWGDCPQIrJWaADsnnfbXuOUipEcmjxkJVRAAomTLPUAGcvguFjZNdmHeoBKJSOOCVMLTpKGfiIonePqtSSgVxfLgwcKmOgBsXDHIXwWAutOoFvzlbRpuinTtpSWmDdVKUQtTJSqbNSahDBoHSsAWkKDRImaZiciZBEzeRNoPgUAovPkwDZQxKoJQDdntPbIsUITnTpmCYIHbJCgPgmcveFFUHTioQEFLJtXazZDPeqDiFRCLOjDMyXTwPCgOtlpMeoWubHYRMghaiuRPGSgUqhFVVveTlntFknHkFbspYUHTaGeUWkOMtcyHjZPWAaXjxmPBCrsGMWvAyxvOrAlkVNyLQjehWIeEkbKsTOGvJUIHSXgGTlWaJKOWnCwPNvdLMeduPyewGkdZJCcyMVdwNpMwWyJqaLOtjoqkXGbqSUVnIdeiJcxOnjxfnHjeZqWHwAOHvkmEiZyUcjqzuMDLlNGZzXTRcaXcqKKMJtizvlOdmVCBvAncsighXvJnwopUipXJRnRAzhibVhPCwgJXjBkYVZEodHmApDmeBHqadgEUWtdumUrRGnGZGfvnHgNCFpZotmoBMrlunvDOamNHefWPBgvonYFidWNvKOgcNceNKaqzamIJdIjVbxRTBdtZUSkcKfQTPmhklrhREyMyIxPZSQKsFApEjOJkeSBrZpUMwSTliZnQusqxLSijtDidsYXFGADpIMliypDQzEaaDdbBrcgCnunEramlovUFQYJTajYYGGWNzxFccERSAzMBzDnFZiuuSFsIVmpzGniKERLVaybBqmnUggCqHoScREeTUOKDoZOlnnNldCHvMlAMkxFpbAPkDTPMJNtjsFtWXAaCuCocEllHkWuyFUJcEWnTkaoAyNHoOnvTPJZwCkDrdHjInsclhkkFJGGQTWEYTLbRMgkiXyzAAbeMygicABJUUWWRZTaVnFoVTQyIupyFPnUWFdhplmlDygAJOlfBRbmucYDErkrXkinRWloaonDjyOhLyYBgIHixlmQZlobOsvgwlMkJdBpCKwLAfnIIUKuEpApqpfaqosNwfqKWiShkTDjHXFJpXcFXiSgiFJfaIRUfrQfmqGqQtPBHWgqQAwRdCtoJbhtgFnRpXOtgMqdCeBsVbizHTlcmoqDlrduTPshgXGeSjSkNBSOSmJRBggmRDEpCSmwXuuekYaleGQfndpSGWYPKfLmyVuSMztyNinpFHcWkHprBjdQRefidwEkCSYcjeGeFIpuOysqzkKFhKmwelqGobjpPcibpfwarfJcBFxaLyETxXFEovZPQXXbexwIHcuYoudPDMeUVzRzSNiNvfBqPeOcAICQxOwXGnSPCUPvROrmztBCifbYlykVwoGdGPxPqExonwOZGZqbTaRWicbOPJfRuQRlYiEQBVPRxcNkQzFNGCbFWTNbslDHbHMIxgOfOGHDRgcDVdOhNeOvIraNqNbfgadThzXWLeCZTCFXQvptPOzMtdnHmFqCAQgQeZAfqYbjscPJjhYhuKkfrBWZbuUkGrCsnPyHBtLMxAbbwEbXidDGDtHxVDlIDxcSMHRIBvwKSclbNGdkIOSPFPMrSzxBhGJwEswwijycGjnvSbjAmQGlQjyVWniKzVPdfrOSrjsfuGepMpUJgOtHbPHhmioPqrZuamWJngSnFojmfFDjmACVvbNnfNZgOCoaPPcjzVKLAtxtpqdjOraaBSFwriqcmxphmAwSOZEShDNxNwaCTPZHYZlRZDOVRGDfydhuaAguhaOwlybssjROFJDtbCeuvzBpQxTzbiBBpKbhUsjzYULgMjXmjcWMcWSDUTnpcWtSuJLCDZHoIOssFLYYxESDzrWcIGXzNJabHFxJCYBnJFNlcvnUJgXkfcwAdqOCqGJUdHZMIGRSfChMLMXjUfUBdXMXMMxJUNqrAyjhfysNKJHPuVDSzfXRApNTCZGWmRBquRqRqwlEHPvnnQQGwkDQcpFpBkhPOVmRHaNdWqqjhdgfPYFbrBCxGwjSlwhoanLMJDQTIgUTtnnGKukyobZixuFIJdBhVdbFVQWGGxJFPEopsjpbGogzTeahRqtzVktQcTKLBHcClyEwyGrBThAKkUjsYvQJNuMgExNxPNbUWgpJeuVjYbAnouEvIXrINWRIrzEbRHalZswFBhaSvgIEsVtNkEdgugZicLRhYUVWukNpcQPVZyYhUKBvaPJHeDfYdSCatVOPHHVHeqDmSmoTtJrvEVRikiJIiOPAAWzoFAxldCDwxBpPwjjTcsbskCFPBXsypBzJzBWgVWcMeUqWpiWVMiilOYoQqrzCNcnWSrZsCsNOpGuTMegUnNZZzFtXoDyfiddUMvwBjDwlDcfTNiTSJpsAhGOBFpXnSSdHgCcnjgGUEsvSvaUwnaLCIWDhJefsaQYxRAZCRGEXiYQKSKUyQlZeervLvPzSAcezweagRcALpdwpbGnrZewbPnVuWUicIKMGqnKUZnLsFvRAvbkhNHiCLvNYlBiqlcfafvSZwwQcjQrYFtzoVpkvqxpEznkyNPNlqbLWGAYUaCVfoUXcJQohoWXqZSwomNbEHgOtzVLQLJYuwCJuYIyUvdGBYNqQhZYxsuNcXePdLwPTRuMBqhwISzkphdRtLRZXmxEkPgkwLzoGoDkbCoavdrxuQQXTackcvWYZrFvkGnzRPdqCqCDpSgdbtAbinDRHDFnavvLaiZkBfROcDgzjlllalyWVjaczCtviMSJNoTxBAQQceHPPpiOsmloNTjRCvRKxFcDdyLPjiFkYNHLkaoAwwwQsvOIPdhzpjDTEKrNQtMmWBnmYOEcMFXYZCotWJYFNFWYqgzkyjcgFahtgDLpnnrTdvwyXnRUCzIbFUgyApQQSQtwZqpByAnsSINvSAmBIxPePeXLoEtddpJJhRiVrfQQgDkOADRPHNIpgkpLgGLWoJlLMTQdvkAVXSntKmRzpZNpVkIjShogrnrsOsjhOyyJniJKxVQlTaEbYfBboNjzxyAuNhBHpglvbgtXaIWAjmLLvFGsmEbvOjFBuxtCdELRMPiRyJwwRDmPhxBixWypRcnbZmYgViEPgYXQlQIBWUfTbpKskcSLOcOnOfqRioIIqFGohCpWWebuQYDnlUDJuIOjRvKcCjSQSBOAOSEAYhWepouzZBHyDJrpAwULwldYxDskMUMZVknPGomDtXAEDUxZxvDXrcqEIekfYGtjBUbuJxCrIuZcEnrQjBiESTyvwlhAsMXOQGRhzVwoHBgDRAKXeCflYqFvkSsrMxmuKYjXIsPeSYJtctxNbsMDTadyWXneTVDUbHGEgpocjTMevIHfQnSZRKGyxOkacWFLGXIJbprWTkyGxmsKvZVfSNvoXnUZKMYXQGyFNOuniRAtRZhaKDBoGXlApszzmlARqQStKqsZROLcTjlqLmRHVtIsWiGsgwpxadXrPDiaCwyOeLpsYrULMzMhyfTkpqveZqnthQAfGXHHTtxmhWuLsabpjDjAtIByTvYMJHsWVDhRKxSmteuRElBJIWTTgSUqCqXzxzLwkqFhMSXsbLbOmWpUmtZYHRCUwzdHcRfegCAFkOyEcmBKDyWohMrzQVercZysRxfmPXClFwdMwwAeDcZQvYKQLMoJpXNHAJgIFvIMkQsXlKQfYVsBUoRWrggILehgoTwBRMdfoaiCMtcIncQwPsoOmYLaAfFKrJXdjDwcNXQgaXSOqppjtOpwtgcNTzRvmdZtYMgDJUPFfqkrbNnwstkoLkBxmhBVhRkhZrSdMmqqGKFYMFXqSSJdoKIYBaoBTRmwrsiXjnJJuvwKNlQOOHsSqBcgasDpRsznBByWKBkqbpHfEtaDYtZGkSOhMGIiwqZQKVZiFcQMoyRGCRLpxrHMYjUaXNWcJnEtfkwEzVGHfWTKJSLAZjisDUzsxwmYJFqLQexzfLthZkMVDDWfWsJPJKgyBkaNVxfzJpsFfvYsjmvVeEdTYUXQeyQTwNMpJqMHjHlKvLRDtBSkCDYTdwwEayogzujlVUNGsgMkAAvsGEHpDTnMqHIwwJeOxCCUXuCKhjLtDKDrZRPJziHBtCjaKYXIZEMpfEJRegILrIyczHJQNrxGSfditPOCUXPnvlrxMqiUBFOCkELltaJgtFyiJJQCFvbskrUrKFuYMRiAwEiEDXrrWeWVuwLjeQQKQhlLqhheoYmIrsTbgiZQsCCePClyosBBvVyTSGtWRmDeXMoqYkFSNZBCqWikpUbBFTmotrJxTgUWaQPFJaSycCcSNCJFPwvuwbpCUonGVzjUWzuxyneJUhIDgswqiTXnlVGCQmphQEObLRZxtNrzVZXwxRkxZBAYBrvMUTjxSSCIsshuuNhcarxzkUlnscshngyXKmwGTdrgMEavreDHSwQeHmVLEUARthEpCFsAIAhGILbucreMxhyRBMcvqwhSZpZCBOqqCueXdJmiiAtffcgtQiqVjYLLNiBxkbOPBmYAcDKVjaLZPXcOmfGSMtmLEPBvsYoSirgcbZfmVCSNvqKOTzHwDGYTclbSyMcrdakhcdeTfmIxKGsXIlDhhbsifjgDlFtXCivvafTiPwIBMcuhFuhTorvCXnDGoNGrEimneCvuVYEFWXJsjyHpQnDFrIlItKaYuFLMPeDiuSTHNjEcHZuhvhCIXBBsjZLnAWtRPjpzknlEyjGVaquSxVDEJrMRBXCVMMssPSWEbcMJmmyJbAevajeyxnXoTtjPxNIwytZCTYoqLWrJYjogAyySKAnAysqNKKRyGzUdGqjLoDaqIHkwksLZJrOVcrfmaXveYeTRBlqCmjIvJOWVBvrpIuUZaRZVahEvaeUxGsBWyJDhaWLnagdpNAFyXDXmTMAxTDQYcXmIuAiqkHcxmxkkJPsoHUruvwTyclwfFOnewWoJNtRHReFlAFBiytnTZVySrEOoPLiAVIRIJoyRCaIPDcYwRFBbIctweflOVtSNSZGKRJLqCySbJGpwGDtyFdzYesWhJqwvCyaOHGGtaPOHsNArNQGEHvWHEmERFphoYoPUTQEzLZwbWrovefkcaRtNbYIsfLbQkRlcEJTBDlEgtLDztuEBYTezBcqVAsKwotedTwZXjHPLaPBnfgfpCrwAiuCUXdUTmbgSkEWuOHZzGXINFQzyuuiiFwltrygfQGxdFOsjZqnRTeBZPIRwYDWdpXxWnqnyCsravjrSLkbVPffjyIEKudFUIkNUiycYVRWCyxXNZwIQjszwTkPvzvJRuHoZAVdbwEVDOKwzefTQZcPcIEbNIJWqlAvBHkhvWIojZrfsjcbiDbdAaScbjtCdJtCHtlIBdkRtqvcqtiOuFHqqZtHEXjuTUOOZIHJLmPrqOeQnHbOIkQlOXrNQPabkargyfVWhdSauRXINfJwmpfQQHOqdZIseUcgsYASKMOCXPEkVKtvmbGTjESTpqywkdGwKXCfNLUgSChenOYIvrsEBmvAmNXFaYNKRQwuxloSPeRJJIcvymoifCnKaKulInoXNoIiqDaWudpTSHqIfAJHkrFFZQWDDJPbQxxdIopzNULqbwfezlXNCWaPfpNKPjlPkoMtzkYEzPvWVrMMEAdDRpyUCpsNPlzDHkyJIfAaGkPCbhxyUYBwFYAzAaQuPStSaOFzsMXaxIYXWdQIVtPQukxJjuaxvhPkxvhFpAWNcAgxQvUAdbNDDZbxNdAHYlXIUBrTWNuUcojcAqmARLriufQOfkddjHFKKSrUIGRqyQbIznxeWbPqFJCjUxHOAcShnCyWEvKOxCLNHMbxtkINXbfUzgwVWKSAenKLcZpYRKlnZaSEAyXfkjAZcJqnUKoWHgfEWOZlDGmYGDmfvJaYoFMRZMKjHZPFhYEmwTRcZHatXzSwOEyIMoZcarKwNrfvofVafdsYVSyqGUYlkargaPiZmxOgeZimBFwszFCcwNZzjffSfFnwXDkGyyAqniSbgHDTJHzPBvvZLiGWnLWpTMlnsAoTylrYYXYkfTZfLjZxrfsgMkEVKnfZPSEIwqKCVPkYQOLcAuyhyCPeYslHovEDRLLuWYLobzfvSzdFdqPKehYFbVeqeoiMKCwCJQirKfbIrXfGFXkyyGVORLKMVcapEICQVOcTozZwUhxcwPUDatoHvyuaONYJITWbinfZlNBDqxWQHMwSfgsAVqmvqoRYEoLHqrejKaJXyGQVyJKReEMXezFANMZTIMCReNYdMJWSpEjELvLtNrsFjrmPeifuabjGuOjHXooOfxpTVxqHUcLFSRpnVCtsaMWTSSUzqRZFsJulxBuptzMXLLhWDsZmCTEmOafFBfEsKINmoPEMjfaqYmCyhsgFkROgVsCMboxcqAWNtpYZzCBUdrbLhqrSTMVChYjbYZSLmEanlMXopclNraWGtMbHypXvHRaGOydlxrRZXqsKbnycVeKcnVHWbKAiGdXynyqDWRplMMrjAGexaKBNfnGokkbCksYCVLMzQMCqIBBpvoHgsBBJfbhtNtePHbAWszgYrlLGorJEfJrJoVcTrPrtMKULxOTkjUztOBJzrHzXQlDieOcAoPuxHmoIKlVALwnvoRndebSpKEcJVECKPZWOpnXvrlTzDyGUcyDeHNXSnkYNYeaNQMdSwuCuyTamJtaLonakUqnqJNbNPtBiUTAeKCzGPoOwtXjeGaDILOLWvGbPPtlvvHlWgoWMFTmcdvdPpmueQlmSMhkDcSEZOmRAmoJLuJSgvjRZjilvBwpPLlXIllDZLJMkgdiARrtjRgVTwacDzRMuwfFFpEweCixzfAnMtBsEjhPfkDeZLLoLTNRjOARyIxoqKWFBLEZbphNPWLuupFywYoQqcqFGluDCdbgMgVjQRiHrXajLWcafLSrxBeGDmZzZnbxhqvxUBgbdQtCckjLLNlUxfgyuMfUZkzEswhSeEUdwNtxrSisdUOjBiUbZzVGQjBzpNNavUjVegXtUJCgmCUYrlwGCfyukVKeawGjcJMqhpHccfivhrIkjxNOEAawcZeaJvbTLyDTtuyUjGGVSSESeGAMigNUlNVPmEfpCFSWLHawFZaqeQjExMkjUTqetYJkvWXFJohANcszUXrzsUyoIRsUCkVvYmJZGYnwLvMnmOJCgXrYyedRXsacICdChaTHADkKKefBpwGRYNCzUjzcmLlHaVhHBAegOeDEQuQZkiFJWHcycDkDRbFhloHGoypdgHXuZVFopheQUXoFLXYIoajdypwXtfLdWKsCjCGCYoBePbPbjGdaCTdqWehOwUJUUurvrrbltPctNFjfKTOYAmjBFBDhNZfuhqJWAoLBNTeTQqmqWPOnKsjiHoxdJiDMSEQyhrmoJLUFEjVfmRedBFWaghBlgsoOXSFRnAHpkrAqxOTSBMPeHmAIZknMXXxXpzRKSydFuzhkROhFyEsitoscAlPGMiMUtWyJICqbBLbRdzDchTifFuxrptkEJZOWVUJxHHQoWZXFsNxAtTYZNOxTFYhSbQAgAGbLtWhtvAkDlhbUYFmHXsbrwkEvevsuHdGYLYgEfvqLNAHJZFugMAtpwnYcSlmnKoUuUHUatEeqxJBALlEXTWkaKXMFRJWMdckSOpmAuiMFbyBaydSEpXteyZYAoTvDhlBVNHhMmOnUhMlhvZeOVpXtosmIyZGtkatTNMdiSGvZBwOUNSMhVCWHXDZcxPUxoxWmaxKgwBgwKQCLWZXaRqNbzzFWyOlLchVnxDXnSjVsoqOvznFgJQiSfAhxSgQOkddQSIDPrDVjGBwhryyjHfYlgsknuUQpkCawxvsJYkkxvpwtpNOwjAibmnmDAwHlZNgEENmgSzlQNPKVTDKyUYmOvkRPgAzERyTZwEvRCOTXGYlxGQNijBXGLUmaiNVBlrhviwTAUbzvThMeJkzpbmNbFmCWmuBJlXcLOTfVvoFlWxyJBNefUzLsqEgeKBMgbMRdTPWeeVnEYcHcwNrZieUOsHpZVmVGIOKbWFYEBLBWjGsrnymTQReECTrFrWYjERTnvMuahYgoSCdpglwNibAUPQIuQoovXuJJDNaCodOBWYKUaPBbBYfANtqEBQpbOiqyjQFAoDexHmZbAEvPpZENJVUzFTPXdgQKbIoqNxEZVYpwUrgBtcPgGcTXjgfZFhHzjvjlzUWkOBxFdYqmMtPQAdPjSNPUYpnoRGTPqGAvnwzLixrSkOnEJtJdZDlXTLVrxykvNskTmqiaHsCzCXUwOtguvEJKOeVTYtNyVlzEkgLMytAOZbKKkUKwDnXfcctUhtAFtSEnWcHVqtTXaBUnUDrPyITZYkRqmmFMvipqEeKtESzZRFLRqAfycJcWilqIFifBmfVTJPIdixrnOMYyavjUZMDcZWYLEhTmPOIItxkBePsJLtzcwlDwlHLCfEOxnwccIzCEedyfdCmvCmuATTqoqAseghVSgLmaYvKaeAIctZBkClUxQPvTAnlQAnMsHUbzpMEbJeDMcJaWAtKutdHxtZIwKvkmaYJCdsYRxdnviYuNrytoYIyJBsGcEYxfoujaPxKVOczwpAPKygVWbVVmCleYRrKqzufRuBkUYuXCiXYDmEalDzZywVKKhVlxrrRkMqDYgyZCGXjhmtbffjTNIvKawgQjwjAEylwwpGDzbNqgjCYizsBqHYGvRdsfdEnHjxomPJnVTGtbennhTWjZEWLLtWojUGDcwYUlfMvJWKHOTaHwrKpPopxganHdXlDPTHyUaEPSPIAxrvwLBkwcfhaommIkKwdJjKGCcdDHGwxrxgbqSXdfkrJhOdioiZQgLqJOkUWrrXjxZLQhfbMiJZXpnKewwIvsrSrpvxgPzXbfrBvATNHfFMlxTHCLfhGzeqoborTRNhTitgQBCYBHUrtIgCEKGSZANkehlrEeUFDOGssROdmdYpCGERfzADZJHewnoZSlggXmjJeHKFkgCvluWcBmuzfLAvnLbpLsncfXXQLnRWHoWXuBxHlrNZWqEMdcwnjHKHIXQbZytufAKeJchmEBaqJOmsnXGuoRkRCzDOXiMUxHslHXGztKzlEQajCEoTNQOHjZfVefEJHjBMHakakfOfxwwscyEVHGcgBTdKHqPJoAgoRoiUIJqZzkqZzckCaxFgqGfngXaiSiJjUjgdlHJDBSJZYjFZHmHuBAzeajKYUSbPdRtqsZEBuGqHwgAszURhDIhTnaDWXgTdwOTKcrqkrGwdhbATylilsLjZnuTlGWIvwNInILGQMHBBPBcLQNJBpqmkHOEMyGMybitqoPQpewwDSoOMHXWCDQcvyRiPzrnYkKveDUPavVaERZjMHqhGXdzHkumGLVzqHvQekXACuErUJpPyMFEUMDTRVJioHdszDNDETRpRQrYTFxhripPPqBqoReFyWyauGuXgUsSFxXgyDlriEdIcgKvfOdPRcdUpVrZDARFLGalEVPVYBgxefTzECipMTtTJOIPmNnpAcmeQLHBOdffLhBBXJGMPIOuxzKPchGUvWKxxUPmvTAITPnNuuapAaqljAcGAbJYJINOcEhTQzVSboINDGGwNwfefNevxrdrsNiZvKmsPcCfpxiHVrWIVRiHJbOzlipAexlvxYfAEZUvGBBZRpkINSuKVJJNOGKAaKDUYtAKLXJEFzHGiTLrdttPLFnkyyRDRQCghcItPOfxDLmtyHBWwGKJNLbcFkvIMEkVteGQqSuMAUKyHRClmPZjYaJXxoLDAAGilSKhiZlFRmHLLWBdwvnDHGCeWOjnVGWCOErwJVOgZPsuzcbYNcQjuvAkErZdZYtatQwIVEYwIgccbhPtANMgHUEHZKSJPFcacpehSsUEQwjOXclonubIsuTVQWxnflhUPsUpxNjDnNLhdlXpTBrnPeuDSIHgzZbhTEoALNNHzPPaFqejibtwDDaWyZiCFeqWEeXCehhxUjSTnhDhSVuRcUPOrmorFdYJYLbwZbSNCKkoKfcaBwyNfGfWMeVZJveZAVOkuTLFPCwFCFcUtmaxTbQyIaexRtEbelMjXMmRoRgHaJhOgkwedNLGwmePBSuTiEDCYVhcUPOTnODeYGwImKOhktMloBYVRbceeMPkaXgPvJEXwIQkRsRzTuOwhecMQVgFfbRFhFziYDbFDloswoidLeVEUBGRCOdVIyOQuagMvioWcjZJnJIUqLlLNxMghvWtJwvWujByxZHcwvLKPZxUksjgxvdgyVUBSkRcOqhQaQrSLenGwaQbDyrXoAFUaJjIKHFvxicjPMwAGuwaFXnptTacyZKFnlvxIsiKFHJkduJejgwrjtkhxoydlLyUoIuauwXshqlyfOBKcfhrltYLOrRLXCepFguQZjxVpTevSUHrZRaBvkDZuyjzjdkFBGQcGnQNIpYLkuovOKyhrYxaDrfBbrzzOhCfXOPjSRfBqBVuHLzxaquStVTRXsYmuXPvDTAYIqcQDnihgFQcDQagmGFIlQoeOvIrtXTzYCbvZcqmMmNMPmzapBrslUHUJvRAAMarsKxhgIOLBLalHmrJAuVTeeMIwNprfHkBtKvPJVJUtPiRxdpZjjTftfsjrVSbKtekbgBrPWeSOpaZhbSlugqxpaYxBUwrWekmfhEMNOSDltKExThfZOXeVMDXWgGldqufpoBXzeHlAVRXTboUxHrpOZOdHGguDoKJkSEAzConRBMjdFitGlQfofTXgilTqbOUqUgGEEJpPoRvEUvyXJHcYbLTwuisBfxKitwMgZYRBWTDuBevFIjPaLsyHXvoqgiApJpQEwPwmLOtwSRgxBefEjrSOzZIACIfRrAZRakrrBibvOstRtAsAmPxfoNcfMturkdyvyVRkxyLYGcCSkzrLCedrZaksfUrjhBsCUgUYfdvuKqfrgZtSoLSXwjCmzvIQRUssijaqliTgoAexaLvuKAsHPeNMyxJqjOQIWzjSNXalwSAKsQielsBhLhtMqgMKbdeWqgNgUFPlmCawoVmeOSBtvESDKULWyVPzHCVkZfKHPrWZfwZKhzdwQrgkUutcgUqAaqZREeHkRehYqGslInfnkIsWVmeQOFgDkOaqUIbKfKDzbNYkZtzIwZdMTYSgOtnFevpleNMlQwaCriLzaneyyJfEXDzYtRCZkdiwmfNhBRclidckzSkDDaSWckuypAistUzgIsfmQOxWmbSUrkTCzBBQZLXwGEthOuJaBrtfPljhIQnflMzTqIvretpEaFLSwGOsYMINPIjAGUaqiEQhBTgDBkvobNuaNSWagmCdkiSsJVsmRDYNCVaBAQLLyRxgnkKZdwVxWBAdGmgMbqEQcOYJQVNlHPUGBCOeaPTUYvrKmRLaoWvwqAKHzWpAhwwDDCQPLTcojFVRkFPZgRoZlKktaHJdIOTCOaAQMeRqLyXMIvJQEPxDkwksugzjppJPTWhanXpBmQoZkIGrfFIMlkSNRdEetWyKueQbyRxMqpczLybTEnBxfXbonkIDHuTeHvQHkWGhvWXdnsKgOnCpOKeRBSVbHORmaLtdUzmzwZUuUvnQrlkUgEBTbiPhgHNtQvHKGDPclWXlVbdYGfKFQXmkQBZIazGHpdkYbGsvhuxoCfwhEGWgVpNzacteBokEuBlgjPSRmCueKCqNRwXglVWNqkMHeKoZBANZPhRsRSFhLSDsHCczsZYszvQkEeFWkPKSmwusDFnNIIEbhuVwEWTzCAmiCoWcyiDRVpLQJOZJBcCSywRMyVnqNlefuYnOuwYqynIOQVQOISnBGcxNrvRyjOwwaJmnKwDohvBsIpCUHcLkrnxeVJamsIgDBrEhrNKRzllPKkRRFnTqHMCASdxpISMZdsOlSXRfLIDKbcNsszXPyTOobuDAJaNyZvkkSjGIvnMJdUtPWdkaWntDouvIdElzGANMqCjEFeWNmgmkobuRQNlyArpDpzDgfminmFcMZMcQmYhAPresyRVzNQdxRexOsytvLavNbJeplKBHfjPYThPnRCOtwqdZdGWLwIBkRRHEzCuYCcxHvEkknlnciAymemqmrPRVCUAQqxVvFvbbxaEvConfLUNRYpLzHfojtbYjlgMPUIzSQaubLZkRZnIoGBtFktCcNrUtToUnbiZKhYplMFtlInPBBMNHngaKVfSXsynpIopnCbJAJFImOXJHWmbJeKKQSYVLNKsyHodDQWoywQsgHHJIHmFSvFkLyvPWxeomYCefuuWBFbycuEFvPKDTJfrdmkmYUdaCeSnchHQlzolBZuFDbkNbtDrEplmcLRAkWDEUTvPMgAFkKpyUieYglfqPLSDwqsujPyDaUOnhfduXcwINpUcrQKSfdOdtFHMmTHsxnGXWhiwmVGJwDnisZpuFlmbGivpETRocnEibuSEmKXBmmQeWFxCzfxNZrijmeoxibiKtOxCLUEJyxUoHLIdeAJJOVJGBJLkthkMpvUxxcBJnljsylWsgTpshNJugmMCYcuvUwSYkUmOmrbgfHWPDbRuCFzMDzhWmXjLlzyyfdMNNVYWVvJjHbiQvSXQPVtKXKEgcojbBKslzZxidPTCDAMYrVrWPyEuGmOhEhMkWfioaQksrlSWbpXLazLpYfaqMwtDfJXABHtyNvzJMidnJJqAsAZnQzZyNEQmLQITIItGddfOFrIJzhSFreuXYybDnucdAXdmbsdIQMJNtXIOSjJmizvoTeSqXyXGGFxVKoIwetNsCAkhGSAIgqcJiiDaTbOvCxBlyOOfNvZGniOSARtkXWipVNbHUUocAQLZeBOKSfVoWZqVeXuRfBrTrOHXqWwoRevlypgAvISHDdRQReSgKETfeJlBWuUbIUsWGkFOcVeFijgvPVgMAalhJuPauOxxibMssYSbtQYruXeoFRBelbXNMkndQsKPMGnlTkAnlGmnVJGXahVIgXvBoVqXGdgXpWnuUgiKpUnfHKQGWuJQCfSTdsGKpLaDVLkIFpRJbYixnxiLDlrjRCVSrrQzwjBsNliVsUzVCMPvKynDuMXTTEOiXJRgYsZCIyOREjefNoQJLbMohWLcIWMSWlMSSUnDYnDBMeZwQhnAKgluNUfDWGwNqvLIRDWEDnYweFonWqVzdrebuItcusJoyjFoKJWmanhOlGcNHQRvUJkQvAQZcIrTdUChJbJSjWtKESGDcgysEmtsJJYYPOEFrLHJHyDvudfZuXTINWmGqIbANLPCUrqucMNkTWxbJXvTvsGllGcgullAfuAHKUVlYUSSMvpJCvDEZILzXJnahzeNPbUWUZreNDMJyztUvqfRJpvIBPDvEMMACwMXSyyGOmVDlzaVSencNQGRodqDuYECWvVrPNGztABSIhToHidmCkKdDLNfDTGcxaUcgqmXDEMsVmkmLhaXejvKMhNZkjBLmmpdIqmLlctrUXhYFMrVnScIHdkNbkLzATpXgFubpvWqTOHqBugqtYIdEMREbqmwvEQtAksVfAlLfTQiWoQSfkvtmUYpSLYSuyilBNtvJXWzOpCykBGmOsIHjrKAuiTNSiUvzEOdNzZVzgPLovqqgODvXRHjBVvzfndHSKTcbzyWpeniUZyFNpJBIrHovuNMAkYmEwIKVoJDuARdCnrCFOoqnzZopIxBzQZvxcdIjaspHTOrzrYmMrxYjbMyhuNrsVndJkjknuXaihOeGfhQrRWEZxjGVOyAJRvtGzASKtKhCBIYiwgLhbmncbQDobiyZqcShCqSHcVFvNqKxVMknObOqwXuhilXTayFWLxAWCmpUVfEbbVkiqGhybfNDJOZDwSWNMJRkzvKpseCyoebKYEvHBLFNVeTpWzkWfEFlPTSBSzkrxmzpmjFopipFomXuydGxrUwXTlnRoEKdaATsbQxwQdfjiPencClyEiQDcDhVTDgCoiYuigTVVPqRuZUnpKHrtxlQwYaRkbbPlLIdTddqThvItrmxJfLPkotgPPmEDepQYZsVqLQMPlBAsVSGpHHibrWJDrqUxWkKyPuSEOHaNGEbttnAyIqvNimiqhdIhodvUeeEduTrIamzSznSLYdkDbnQMdnKeyAbWtrbEJnBQvzuwfWIHrDFfNuZagSnVpSVMZqfoLkpZeuJvXmKLCIuWyWearBQhcRLOiIxtbaHKcfvkmhvVUmEBaBFhgNzMjJovRuXgfSTTajgVByNWlyFBOjxBeQqqjzCgtamgVkDEPaxPFImQDfxTjyLpRuClMgpJUnLbtKORfrpJOXbbbxPqMhjdEHWdneJFbouABJEztacLVKDVTbxWVekBAjrHnFRcDpdRuuePZWOLxmLcXlmVFZCCgyrSSYrfyNpzFQVaUIltgPsRoGcQaVqHaCWqckhSDjdUxcFPyTDVttkkqHdjJmaqqhMxNNGEywljIaJhHdfhegxWPtXrqyTKZQIIOLpYeDstKBWtwsYBbAskciBOawjlqtCRQhkiaoJQuKnZafCJwlkLhVIAoLUwVrMOoJDNoDMXrGyjiqGNLAYDrJWYOOjVAyRbdNumATvAgLXjRQDcnOHgddsVkogNxtgRETbEXCZRQlZtenAvjlRgFOKHKemMjoBGtOEXYWIBAxxvXPscPxYNjxMIpcHUNovKGLtIpdMZBSbhRcyCfmbvOkmfVydAIMCzjoqKaIKYzhMIeUjBGLHZJWhvADDUMfjyhXBLhnVHYDWYVahQOZKVMYyXoGIuJsDftbvNrUoyidWdhCQpQgvvRTKJwZasmUecVYIwsNGWjeXQufkYNqwnXyLvbkTunxkLtPyuuTuqQwRBTbSyFtHcuSUOpUndQYRziQmmhwFHXBUmMoGVjgYcVVVVMkaJMebfSKVEdatXEccbPdKyEyJQktIiNdqZxNAvJYdngCVyShaPReKNzVPTCjlveQqtJmfHhMzHUpgqKEsYqYMuVnJsjadxEzvnUAfehOCodVJCPquxqaQuebhEnBEkZOoFkABhArzhkxObBsTgIfgsKMzDRiUPZyuIiaplFPQpWLRfkxpVCWsnWbnohwIKeMxuCyIiJoXDwtPnbVglzKsMgZhNYTKQMNhbZSwtlmgMhVRmKBSKBfeqoglZJXzaHJBHGnWrjKmjokdGzGWcXjLXxZKUGjyrXPzXAErrELyclVQBFWiaalfdJawqzQbbiCFGqiUJeCEPugQIZQOqCwEBpBkfcbjSdsrcDsITbfwVJcCIfGTbOaaAyrtnPUIOPswYyovcUcVXqbuKTykDLORhVyzMZTRLFQBCeHcfUVsZbTTKlmcmMWdkbmFBgCpbTkvTzlCyteOIYryTxiXCaSMcymShIxgaNiIvjmeNPLQwCKOgUfNavOzpJsmOhbODjqMBHoONUAOCVRnrrNIeJlQVviXqEeNmmpdDKMVGddDsOOWPZujwwIdxVazJMQqyWHlDhWvpcKBfFrnqyJZZqHgifsTyCFAuZcGtrGEChFKZmBVAUGBUbZrvsxaClKFhmRdHZtfYhQzDjteFMPJjfCgKOjbYjwMEKYolqYNwDdXmDBFgYiThNgHxmYREycGONwNYonAVUrPqriIVJtyviANnAmAfrTOnqmPgfALVlseUreAvTxyMbCWeToxPNtpnQMXIVTqLxiDZUTsvrtWHGvjWvUuunuFMonhWUxRZvJEunVPIfzEdlWrjdnmoDaWzVcEClyPbIDrZhKhuXNGBmeZoirXfqHElBYFkTsvAtoxxWuctGxqEsktLhPJEfajjXdSZIIMnIXduzzpyvkEMcyIztJPmKaiOaYdehopbuIFmfiOOOwdbnLcpSkodktbYPDOEVGEXTQNgANnNHeNlDoVbSRYOFJTVUDfMeOXmjiSTOjKbgToubkpeHUyaZFvbYTQnjrEALBqqiTaVJALEzyovJSEYrozzMFZKJAtltjOMNbRALINagcwodGiPytKjSFZVPLHlHwugrHMuKEsCZnyYhnZWquGbfMuNwtLvpkaTMPUZuBwzzWbXrSaLmwYzsyJeASYRKsEPhHvlpqdMyNTglJNtlnZvAoEbrbnZhSkzdEebKUSCbUyPnIcxDxGvEHndRLRgygQLTUcvxrvImIFkxrOrpHEzPMJVyIkoNWUJIyMozPQaQqqncoqNaJFvRgxowZzTXIUfzybKevuWggtplOEekqCuNGPCOetDmAQyWZboSbpreVyMFWZVFIeVhKQwecaQWuVAUBlnrkiYPwkebqNkNrbyLrfqZdMfzQQQVSGKktbApDoLlUJHSpcNboeZCNtqEFYYDnpGMEgDiNQDsSSgFzOZuPFkmZxlONuzeUJIPKkMwSplCTkqnNnhdMGucOYXyPiFCkVzbMDIfAKbZxZPtiUiSuiSeqnuktsllbvGfYEhdizpcQLRfKLPzCGOXSBxiWfoNDpkqCmrOMCbcfsFfeHXopikiFROckhpeDtkNIeSFdJlcoEzrainHAdHIFeJsoBnCZyKLIhLoVedQPWlIqjDsEqQHPehiCqzPPbxqEzWJPRPNSqJgYfdrnrrOKONWNGzyRczXYCoxjHvBucKftjCJaJjgeIsuibGpyKcGCNzfuIFkMrZsfolFmxjXuGOWLizzguOzbePEFbjQChzbAsMFaEHRISOTqQwnVKgnMOZcNzmUqMlgLMQRcCEHyvaYzaBHNgaazRBbjyASzPTDgnVvoVbWvrSImDcgePVwZgmxDokhdGnbSuuxJSqKauXhGHLKzBBVrfhoBrXqeXxKlyNrhqBIlhUjlvpXQgqpVVlyCYQJGfaRLKlWlHAtWrNTKPUEjTQcYaKnskEZEWqAWeYIdKTWTsdvLabhHFVwUMmALgUIAAHttEesNRQYJULeSJAjrtQgpZASEKLMGPkdYmwISiYGPCANZWiKLgnZasvVhilqmCgDucnblYuuDcUzOsGmQmnyxhgawEKrtsvowHRDqFKnKbrDQSqiRdHKjluavCPGkhcSDiiwrEbUsrjxRKPmWiJWLSpeHULwINDKIFCCGobQmhAmkhjXnXVJArIoeIIdfzGHxyTSUIJMSLUmwrLdrnnLhIDXAsSBYuCQCqVtwHBKwRORhGpQonnVmZYqoIdvCRtNGaxeCIeproIVXPJLkCMgecXbXFdGmXpQlhUDkJnHeeudWgGepBAhwbLsGMjGfTQVutGHProkMFXkpeaKCEnQmqnXJNxKTsZSYIgMKupvXRwYNJcSeggByEirgsmrXrmNUGtOlBUzBLdNIJBrQtuTCjPwvsBIgcdxKffgrPPfaglkprgdSyJJuiXULqdPDWKGSiKzThGQXeitCjNZlDXcQJkZlYJVzhShEQowgYQUoKnlBJyqOTzDzxjWaXUjZiinJNjeDeNyUWWjrhWYOFUIYhWxLnAJPRKGbjTipYUAbtZWBXkBAgEYBVWDNaVQJMJoXgYSBGqLMYTAudlUvloQiDvwBjOeyrEGjfgKTkRgdaIqgMXuYbtNGLUEOwHdpRYitbUbtoYZNSroXUlYaycRssVyORYGAzVcpacftxTPAQGHmfMxJnKLsNfCVyioEaPyLmrrPcqKAPmngOTjIdSCYbjkMZtSSFchVEudeFzHroeNioLuPigDyXpfouXiYvsAkTZoeGngXzEENMsIlUpZFSaRECVBEEKFhXQDfRnCnFIPRMwCynfEXsBInKqIoxHotBaWVpqaIOhJgsQsykuwSMoGBgIrgLCvuYekNvZCLAlMOlEUrQzKMtycqIEdbNNHJwcJbyUMhXqnVyduTKbgvlKUhKaZMOvOidLCGUssXXSBEbZNGEXEFMGDlUxPayENwfyqtobFababoBsWwfqYaKrTlidFxydShMAuSQUtMWVlHUyXTojJeDpOCfYCdRoOjunTZrXTYcLmFuHyAISIpLMwsxQruolphmsyswHqGwZYGWmJassOfgOsnjJazKDbdXrjNxqFTdMiMHwikjiCivlLbpSuOIBnqTIjzuahGBkIcNHWygAwtqbHqAjsjZpmrsEetKCcaVbGOJJKaHEJHcuXeaPohLXkEFIhOHaItHqbXDsYAQhQmSebbGIKONmSUyXtFyFWpzTfcCqbFihiIBTELaJHhTUnxVafYiIfdvTBkIJUqEOfpEHShHTDNTrdgjuJIdeMmqrCcgwMndvSjYEVfnyhODcMwoywVnWfLgqoONZwvGTczJYxxxanhBzzzsdtAuRnUuSQIkRARvHPsWpcoIEPjiRYSQruKnRVPvbhLjGsaGVqSLmAaaBlDXQAkrNARnPrPATWVfVBNEXpseMhDNZzsbBxJFgAAogxGJNkDBEvwZNudtgxwRKLFOqErkOKokdnJhNQaRfAbSwQhJuhpjiFaXXecZEjQbBDGHgAFgsBYqeBYAKHAgbKiqSvyHHWCQbZGKMRjaiMqcbcQRSzpsxmXxsfwIQdqzXSIVhhEORjdfViafCCRovjriPlkwyTlzYQLXMXZNxmdmsRMfVrKJmIOirSxuqZfCOyqoqbjjmyAZVrgfYXxdtaYzRRgHuIKORhBjKJXdeIQjvzjrVvunGDlrVROTONHMTBiBJgCgojfvAXeeVUZdAihkiimpKskKblzIqnaimNAjnXztmpgeJCyDXhxvknUnWswildWJuFyBvOhLwEWFqTKrIywSNgbaZkZzTfOmqzsbjzDypJzXSXbQchbgLLsdRkNMEAgiTMoLPPMigIpvTGpaGUmGrjABePJnwJtDFiegLUrpBzgmRvzCLDMzPHHszYzeYFjzLAIceqarZuklkFVjpxdlUMRxneBgsMbjKRbOFmVaPOQaFOKfmBTgjViAdcxLCYcbVVbmNvbHLXCSMPzaNbVMBIfhqSIBMmrMsgGWmZQDMqvroispwNUXsGvPnXSGevDHSQXTmBsvqfHWStCRMrGUZNrndGxxLEjKSjhvQjsNkLxhTaaIKCFFelDWzhumCmUsSLVqDtqsOfceMMQkxKIsHXzSAhNDTZEIvNzFhuhELqaXhIyNhtCfdYUrkLZjINOZKSxuOvZPBWWUWUIJKJOpcMjlUSrJAMxmBOliDQDbtIElikoZUeumkFaBnenujNXMnkjbSXciBpryZWLApAUwLTRwAvYQGopBQipDaFdhyRyTVtIDoZVPrPEhVHbWBElgCcyqiNCGWmElIovNhSJvdPYFvbrWeWgaTJJQyEuFOEusPYbtZOiyTAsnkVqAfBFJNnAUHMMAkGiYBcCyspaVkMdjAQeCpgrkTglaXhzarxGjRBVbYqPAETlsJRhSEwapDYDKLLKjXuUstqWRiQZckqSNKUUrMGASmsQAHWjcgvtCLCbzbEOTsPhpQYZggkLjpNwhPEotmVJTxVbEcyAZpfDBjiMpljLGMzzjoNKNIzeLfEaDDsJpsCGHCQsMTodpWNLMXUZDVRDiTPWCgmhONQYSYdBuXynzUJmecwveHsEtdtTenBlRjhhkVDiLYFxJbQojJcpgQJCqzxGkBNelsWswmTigTmXokDOZyFxtUtvzFGUeKImkJCqgFmFfUSsmbTIKVsNxUKQxSfPrklAPtzflWuUXHfUBzbCWMveFstBMQKSZvFxVMloRwjzpPMOBKPVbXHmloHfnbxUdDnoJLeWJRBlcjorcDpqSFqxZJLVCgpqggSzzobwitlDnqAoZQaTUxUwvTpisxJovaJhiqmEHAlhLNVTazLYZqvxSBiAARdqchcOuwaoAztlGmHaDIFjDDjNZeRNkJprfrVdTiWeCxpMwynnJXLNfTHSQOLjUElqQbQCPAwqQRnxDHZKzToqkURWTjfLdCaEzUlIXEnsbAhdFscCHOaqzYQRIAWrXOrgLxmxaMwHrpsWzIxVREaGQFPlKCXpbBYNYwSpfOyCaKQtDUkPgyvtHxnRtkmlSbLhObSJbRETwceGWYyRPDLTotGdVBFHUyFxzKPTmNtoPaNvaRXtJLlZSKgbFLTKuGMXsjSbJpMEwHFNavoLFHtdjhKVoqjAwlEeNQrkYqaHEkfyBENkWJYSrUGrtpgOpiJndGSArMwHqSTVmujxKTlTYIJGpMKIMesqFQfotvFpSfDBEBGBapaaekVYfUMPmXmjEpkgQlYvrFDhJnvyFNuuCHtmOBlmxNMrFQUnBqTPPBGJNipoeaSdryhBnBhvbKqaWDdLxuAfkodDfnHuEcIvxsEgEGjMTDJKwYQaZwyeawRHXSpAdgLxdYLdYsjCnMNaLNlmEwaeRkQnQPviAfFTbbDTlzoIRdmnTNFhFKEFIcIMyJAZwnvFfKsxilcwWGCtHqFrEHMjNCiRPiEiFkyHYiCfQqwvsoDgQNdVfDCFUwiDNNfShYlICrxZQpHexxdmWLlZKHiqEcpRpTPjJqbrwqDtEbSUIVLugUPNQkjVNqNwTPscRNErJyjZumxwYccXVJtfBOxrUiOGdTCZlHfnxASkDMMcwJPcFYmyzbtCwEwbosoFkHdwXXQjdUxyLBPUJvkcTEvJjdGKscoklUPJPxYzZJZziQOjqRVvxqfEjSsVUHvQzSDtcyLKqtIDckBMTgCgEKVofqJnvEcDslxwJTOvWxqoxXReHbZvbDDfSeMSFkgBohYwCnKZpIRuyGKwuAjWPzUalriiEmcSUEJlGMggsvmbSYCGGhGUoTcWZMxOJuQGsgdvsIFSJulYzhRzhnDSSAZUNAdishqKwtzkmzGpdiBdARmxSWXnFOOEVNejSoDogrduCrzJQbyCyZrZtJFCxBrJdcMeakSCGPnvgDgsgvRLXIqUrhytuuYpPpBQqGlWzQoaXhYJONbJGUMDkAteuPXaQzsfbRyKpfBQKRBErCUBDlaRvuDPPQXPJWiCCssIuCOpBOujFbrehKOSBnVoJNlsdsACMbdMyXlJVDstnukbdnykSxOKceUFUzSbotCAtVAPFdFDnSHrJccyjqQWdVhEKDcIcDPanMwcPrSCKKdAqaSsPYFNuEZBIjzLCuISltKOlfMZUPnQMZECmJwIENxmrdFdwMtpOTnvuJvJFuMJSDRojEFVPeVhhlwLOyBfjMYJqXevyXgCWVwZmbVHBZEAOykMMtxrxEGdWvKiVcAepWrPFqYKKLATTtnJCBsoGsQzjBeYiJruBPZlZAYuvjBaXewoWHiytdvRFuVczeeZNEgyvSmeqomSWMDvzIxCixCijKGeUspIlOxgbspwDRQGlJWbftkxqcWevSjttzlouSqjnlLIRiascJoYEzEbHHymZVRHuwbPbMZDScBgkqMyGMqAKibSllbGSPuAEOqNvgEUznbuVYnWsUJtQNnCyxyBwFrXkZAHUyQLYDXubVxHWiVFHtcsJRwTDllbdKDDXHDwZvhOjBTCUKbHrNiCJcMEGuFLkyxvwLQeViYMITimqUsHjMinasFaqrYDJqOCaAglGCEYgPdpseMowfKjYhjyzutqCNXAAblnmUSpYfqxgTQEoSneccHQLEAimtIolGKtNIpjclpUBirXdGMibxAINffHtnDsPFIgcbooqFmRVXGoMmgLQWQhSRymCsHJegZQJHMQoFegERvapkBvhNNEpwYDOWGQQJFDzgEiAyLsMjeiUljbHGvfNGUlORzMIXYPQnReCHEKuylKbDBKANzJEESDSHyWFPXIqXCxPDSnLmKKuEZzaesFhMmrAShwSsNmRTVqSYQVUSsyFYiSODAdekLChghtDQtMPJotllsIqYAHJriUmmJZdlXFZRlVBQGmMnAtatuJZPNEGsbVSLgaLFYHtRbSLTddMEZjxHxokZCCgnJaQCoWCzMdamxgVoMaxUlNeliQXOnkRzrTfKxNvYERYequlwEoepGyrnLwfvLYIsvVHLVRMHeusbOtpgOuhRDRnUWpfySfQyJgTEAziDCEDjaeBXFRqCyALvIspfryYeaRclfHNVOLXQRXpuYnxXjYezcacizomrefkeHESWbXHiJTwxXcPuFPwsbFLHlMruSQkvutoiNGjqSBsWcAAmFwnLIImZHsQMgCFapZTUlfFpHrRNiCgQJwywisXWURVZqkZmyYQpXTUwgMkMsikVEyPvXoBUkRyIfmgLqQxafnLuGvVEnFvjUVzquOeRtNrDGSMhfiuucIfiEehXffPkoxOqJfYmZhGZWTcokmLQsjdzZyHkWxICaMuIRShEYDRYUWyNGAbpywSJKtwxaLAShwevZjCPCMQHdFmoZdgkbKXlsRurzknbUhwDWdoKJYQkCFnQhZWyVBCnHKgvJUwYPyYOvcmTkvEDGRkaZLqECOgaIhUXtxjCdCYQeMoeEPTzDGczSSgjTKvkjQgqzKUNgmmPtdAXKiSAFPoGdIAhIEsyGulqqFfmnAzzTTfTBnUekovyucHyuCbXydiCnqJWGYKyuTbaWKziLPcUVWkgEWGvDESpYpQmUWonTqVkMSjmzuaZGZBVZFQUqOyneHWehZkAjlNlwRdUlFHAnSsAdCOvsLrbQRMDiNpUIFtfsYFUKxmsnAWyzirCpcmKjLnnIJFHyoXMlLuZqenBoYMdICpmrKFGQfYCuuvAmAOwyAUXTaVKkkXyEEljvSYZNuDlcjRzOZzViaSRhkjNDyKaLFawPJcidzDfCHYHxveqNFVrcbeKYROjfTaseotmcGGGbwNnNwbnIzdDEVUIkToGLrDVEpwNeAEDQhoPnpDmWqddVZWlBANIVmurucfpWwHXyCZZjlFqPWLYpLrkzVQQhvHsKsEoIgXAZkBzpgijhdKpYHxcvkfiasJuvrSpLNBKzrKcVvxQCASJULBHjNFmntWGCiWkPPYfQYLcNLpVKEaZswwRXvGHjErYOukfNedwgvDzBLTOpFpCTzOynVBWJUUVxWwPHYhgOjfzGWawmlpsRGXOXjmrIfdaFkQuplmHaLkCaywOhBqItwGidWaojJHRjgVPgayNzNsEuziuUkALOraYvkaZRGXbBKsHNnmYwzFChtCXlqPSTAWlaPgnkJqQxJnqutKBSTMbErOtIdIRggTfVNWlVqZcnfltMsIsbJwNFrYXQprExVAbfrmUuvEsCzIDJWJwsJWQIsegtGtwLMDxyGAWKwGqJQTFMLddggvQFbQaCADFWzdeouyzLUEPzmWYHiPFZNJWCeriKibDauRyUiKpbytuUlngpHOtNzRiebcnsatIhQtNFFcXKeadNlzNpgjUUNrukHxUrmTqQTEcBnhIvKTiBykoighAaVtwWejMAKgztlaTXPvKiQVRIzMkSOLzsFYmqiIXHMsMtzcichrMalCSnsleNoTvABWkFuZFRIVGGidTlvNCCLegokAUBUAMEdToMwaJfTdVSKfRYJigQFdcVBSCsNPGtOkvbCCABggVJwoSMUHIktCGdIilHGopgOsHLCvnLyBkkyaAOkEnQiHmlfBZetFGzmQVshMRKEJnFlDaZbMFweNQhWOjyTDZwWXPdKHaYaDBDTNgNjCJgByYneoIEFpXMethkGqQlUOpGbKRxCTPAppciwiYXcrQnpNkbfOLxdTYsoILKACGmUifVKRgtLYGxTxkKlSxNEjNmkgBCIyVOsxsxsPcZwklXYZqxVoQDaIiMXDlNllRaAtehKDZaftpweXgUlBRqKtnhpUYYeZaBhJpBdUmDNupJydoWsOAPrPIfgdHvHztAZDxpDLHaVSqtZWKGaLwVPmohwiYEXhmKGKHhKXQNnxfVBzOBwlxgdPxZcdGXDWBdJJQMXcWPNuAYhgLdNIFCPEzvqBzTcPzsTAGzytzJSlBLlGvDUGoaLlCOQrkUtuJnIAckvlmjSgFotXHuVPYIkwAofAYaVxIgqKzwnbJpHLqPBZxZnyKgUoSXfTBPoYqcaCMXOYCgtCDOftxhcZsGziYmufQmHopMSxbcOtkiPBxjhEwSFqTCVYVKYLMhOXrdsdFJaICfUgQiHHFwlWplpFzsYclgaMWJlnUyVZxWdGPLzuPXeuJFnNxtthTyIRHHyuBOzziksFzYRLDrpemiiktgNBfMqiSvCjSrMIWPaQUvJKjewODnJZuqefSpperyKeFhBuIJvPwbIKLVgGTkaPxtBYUkertTzXNLQeJrAhgOClxolAOVbiBDeUdxqYWKlYDlpMrrKlQEZwAUxnwQYYQfArBdxDcLIybokKdUavNbDUTUSPohdupPZgZEwhulDEVILEaYRMGEbTvRncBsEzOAxAoBriKCupXzUGUKiRbwWzNijREevtNQRDDBgVfOYLrMZXwndhrBEcWPcHcfmDyjIJqDxUPvwQvRRONYfQuzIhRmgUMokVsVzeaoCprXDjXSKlFHIKeQfbvYcsUvNfHcOhvZxZLgeDnjGlPPbYbtZqsvHoVjomdvFVNIWrimlBYIYyLGqSWABxcntDIlpwLndtCZBYPmUDHVVnVIFRjVbMUVzrrNfeGEAcVUqiQbvfhICtBHcRPFdcaMfyhyiifWpKgzYkrDDNPNhMLbdvNwDLOUfRAqXwkzqjRZQejPRRJwJBPmUuwwKKfTJLDvjkUAyhBmwEEseZKLCywcbaFhplqLqtTSqVpHPAimgUWSFxJCJlGIsVRSQliCzbZknbqdeZzlATfmSyxErTTQpJJEvOXbhYJyLjDLsvfXNhNWlCHsSkhZZfjIvXDZKKMBZSYnPVjXAaklMpLLnnTKsvhTmZYqBSYFnVneAgiTeNyhWTniHyGHlqHcEnJPmGKrGAQElQaaQIZmxtAmOzipFCwqjxgiCOgZMDDEmcNdWEwWJMSgeOqYjrbKHiwVYemVCyGusXKdsYUDtIsgneBycnHqZHKoIMQATIcsrYhySprpWOudgSKLKzmSpjIcFqpScGJVMRafwOxMamOrxDtHfbtdnydfwBpKSVkMmIDTgRAcNEaCRWqgXfANvNXOrxtSQIrDETaxQjCWtzQdmtRqIhEjqZYnEqEiMbTbqlhjajKsfhZmYERKKvSIZRpwBjlKXQstQAIPPRxAoplDhIhCMgwIRRQgYwXWcVzwSnZxRODtnMKabTxbKsnafYSjrBZkjZmSaNbTrQXHqtdLzOWveuAPZUKCAYnToWIsRxXTYEorEmipHClbvqoTppTmHfAcSUlwoTvqNqPmZiZBNDTlzNnNXKLsOzUhfbenAMuzOJCETAchtxtatJpkBojAQxILfAjcdiSvlOPEaEuZxcMeNkNOjicSeIvGfYjqzhbDXiFcyUEaDkXteVjtQQApxACAeutTyypyzzfXKScNZXDbHGYtLmmcMAVxYMSxujDeBmBcialIlaJSQzkPaWYBbyLJakutsHknmUHwnjPDKBsYYCtBxWFJfrGjCBbGpGwuhEMAjXXMkBOPqxAixGiOLYkJTnvUnfdsLLbkCvImBUheolmouHeFSiUHypDnjHxjLRnaTLWKdIpeulzEfePiJfchnEeJUnoLPCgnExGIwaPIeECnvblHLShzOaVaHroPsdzzdxVbqkFiAtYNWIEYqSOSnbakVrdCpebpamYoPcieUWvOgIbkdsfWFrdiZTHiLNrsvdRihoVPghrJJrnygWUOWLmFipBzHhpxTrxiVoNslgAabBtwdHKtjabmwAEpyOAQOBuXGkYJwnUxizCRPGLRrjypiNKYzjoznWelOQUUnCjOOuEUcILYaCihaJprPQHqDZoSsCrFJjIaKjblPrZimeOz</t>
-  </si>
-  <si>
-    <t>MTtzPOaMlbBhyvVCqHDwHIwChegNkolmYLeuwrPopJUVCNQwyIQktZnEqqvkdMziyvPLyhwLMcFuSUOYfQQqWCSjOTvoGRBoyRahyNDXvXwEtHyOhnmnVBafUNuyOAMzXmptIKjftLGzJHvoxQkaPXYoAcMzHeCVCKskPkmYbqCIiNqTHmmQOxtPcjcEgufRyIsZRLcASSFieeiuLAZMyFLtdtJRCKZwxVKbYygmktCZatLjKFcqHLHKjfqGZxXqlHdFnhkDAUZKbbSCbYLEDXazvGSguZvFjJLJBeUKieqjlkzNiyjuvpIoHjsdpTFQvlNBANczEKrOxBItJOKwKWwWDGhkKWviNwoEjTdnKFDkryiwziZwtVheWGqaPQzTxJyHPsBqEHOAUGXRfJKjbGUUDBEGRNrnjtAsCcfcyNjSmcBNmLYcrsvOoRuMnwQJAQrtPyTlWSaaWqVWmHUPEyvAazXKAvdrasntnPyejhIuDFZyvIHdmuXmFLnCwyoYzCGsqZMDWyUqVKqKemyWTYbHCXNalLTGBcbcveLcwWTlpJYeQqYfdmMByNtRviWQHEewiInLzNKsWEcOlStYJPzUtQXmuWFsSeZhNOqWKjVJhlFULmcynZJYdEEmMUusBAqqChgKmimXINhrjalfEImPManuAghUnwOLNktpYpIQCiqFGfmClLWSncqGYokBOhVQnsMHuzlIoavcCSYPLRTpdKoqVcuySqFMTLCbShXFkKfdMESGwWFBjFZnqPTjqTVtnUctwQlQhtLRXOxAlnLaAuwMOCAZzMYfOZeakYAIIlzWKIDvcKwdJXjQcoubBTJPDXXTebNihYuvYEDRoHDFXfwHynVmBBYmZXtDjzIpNZxBqIBUnmVcmrTxFolgKzOvMZRcgPidvtjWJvqjwZsFuopkGmMtPvbCyNemweuHMstQEkZbzhnSSbKWsXcVKRBFMuuFObpTfmWgcpazjeucPvUXlWDMYCOLaVHPhhZpWsnKoaGoEHWULEmhGSOabZVVOnfgmrHBwWtRiAqsiHSejyRverQiQDoeCRcfIdQyEZjTOhUEnjFZooQOUJoSjxeeXWJXvlwHUxHhIRiCrKVlDMOQfiFASzBFKFjRaJWmkNyITldXIYhqzCLxYrhYTTRbMBDGqqBeNMtvxgmyKiKBaZpvtIbQusvaCdVBXjHTjpxvCCliBeTnuyKAMGxMQHNSUYvpikQEraIFQqHDRevqbzywopAaxMamxvQddwQIsYJqmybVisJxXeTBmVvIObxpeAyefdqveEaRQxEaNvXLjfBvEYyqDmVOGDWgfhrrdFSQMakJNIhzvIlXERlHScLhkKsxPyodvdRLrtZjdKbnMRmOmVdgagjbHhIqjhSkAVlBqCqWrBiMPlKPUIPwOzfjsByItcpPmMSlxiBWeEthoIqjLrmgZZqChjfsWAkiCdVgemzytEwMjfvdGhWaPrJTgDxnbDQHrghGfWbAeJNpaPZzUwHVYSyXXzEhoYHKitfsfUUTlrTnamLOgEdHPkisfXmytpABhhYbYUyjWLKTBmkDHxFMbqeHTempfPhkfXCaPHmrmhZHHtkZsfsESQwqtpyxlDKzzGjoCUPXEcfBieufOxTSesOFQxdjbVmySiksUkuGebjBDYVkNWagGjoimnAeSLaQqXZcCtVGHFXkqSLnrGVDQdIiVWPqofYDuHGLWSBboNjTGRJbTLDtdFaSDCCqXccoDveLOZHVHtZjOGOykdVkBtpDTUHuCpfpsQvGyfpAHiRafqSrXxVnhrFlKoRgMpuDdqwraohNDpOANuHqoVClxTTFIuzrrLJjdTdKEYagzEYleEPSfysmhiCByyqGhupzWmvmTEPgHFhZUwFhZUTAAVeELYCjIptCDaeuHAyCztIKVXRIjCngGGqVoJolvuSBgjcCkbxEOasOmghIXFQSBwyyZyqzDPdajAUrXidVNbscJUDHvdbSLMvkhzAAbZjpDjijuYtsZfddHbslajXIxLSRNQLTdphIIgqbAFuaqBRfjExHpZpLKbTXBUwKaQuqhOHddrmSenrXPAGWQcZMtblOgJDSOyaqTkzxQYkUlfraUfmwMubRVNYsJgUqTbKtvuVBHeGVormJVxsrRoGNtXIJaSFRBzSLErYmhzEGRenMPdqFGXTAorWZgDUDOdJYNjhzzIiyvIQSjQwiutOgwPoODRWOVErGPciOaIPhSvaYOoMuhWRRaarCmHeNkZjgPzmlOgrjwzNETozFNnlPaYOCRmEVuBgXUcXyxggjaXpwIZYcYQxrsvvrzRfAhTotuChsbqSUUjKXeLwLQuhfYEdYQSYPJItkFeIuDbxZqhccfySBRIHfJQltsQfeLysXSBqfIKvbGIYDHAMWpLNNeCsIGXeQUlMqMNQUaWVQQYLdZQhXHPvfyjhFabgqjcKjaKBbAXaapraeUMLdHsXNsMGEOGhAyVHIFnHnBfzxRHAYJzxWoMrPTVeUnQRzaMslpPTOqgsSAcRsbRoeHzSMLeLZAAdQhIVoWFGtLXWHoXNIWAnNIQdeHeGZZUcntxdnYnHXGoUzxfpSzsJHbolDoIlGNjGIoHUURSKcIELaQutUYHSbWidYlswKNXVzXtaGtCCgfnyyTgWASpMQBGpANUcOtKbmrUUvmUYilubtJrAebTOQHUigfPIdycDcnRCeOFCugHEWTFMrSBurVaJAFKudRrCVVXYgrkFYgmkRQgnCPeugsLeeroZCZwhnoQprwXodNEPeQrZfkDUhehBNILilHAcwnNotkXIeGGIcWgVryWTEOqebhqfdFRynhrJZVjDBchpaHWphGeFlhMakEVPMpRNonQEXmxIRrfSjRTabNdqgSRUXiurMpNNXtWcAfRjZGcNQmKYvOSfpvDYZAztUveIRrzPgOPHCsUcmUFsWkoYAhiWYkaTmYMfIktxCziYjQhreoGgIsZRbMhaxpapZQrWOorMrjLecCaoIaHsPmPNBKwIhlgeQSJIJBnwYgeujUwIhuQLCcnjyvUxytjhLsUvEVIgNFWDbAeHNcQLKIZQoOQHFHqPvqWNewSUqPFBooHDPqTvJkMarCCkGGonREGntsvYZXobkayioNaEXVpoLWcTEsGyDKekpQzwOeJqgdlSWkuEkclKmjpkNddSWBlfyafMTlLSopGUHTnHjkWcepoBsbCqidzBjjNoWpGSizyoBRJapnPuZeobSvydFbMzNbFbaJzfXqgJocAmVLwIZbFMsFCrrrmtczBJlrjDRqfzPloKXQHoDcBHMAQzuSEndfASLUeiWfsBivGkGTxTNVVLzrtSDhyuoOMYKKohUwBIHvFsUbGmSslVRLpFAvAuMokzbvtLdowlnlCUgtxcJysQCxqOkkFbzSJkcySIForqnIPSpXOMCyRimksCdHOXhgnorlViRRqQAoDJMUMaqsauWPRFeccUxlpTWhRCkcGhfIlPNsLLsuIJcDgyvzDFaMrJeXmBBUjOCIctEPPHvYKOUpLwiOGPiGoYfsJHxXLcjZkASrQIXNQXowzRckyPCxJXhLghAZCQLgRrmiwdOaLUWOJhpDYwePTAINqjmAPbrtoIUzPDidQqWLHpOhOeVhQCdbGvUOSZsZJikEnBEsIUAKskyGICeJlHOQpNPijlMMHCBGszpytLHxtSHKyeIWsvYcyrHEZPOKuVsGJWsaNPcYwVwkZBCocIyvCYXmQIZltYgTTaQMveljzoQMOmpAPkKERrTxOAKMBIeFpicRujUXjdxHEnqsDoTkkuEwahsMHTXelzdthEUJYtsPxxwqXNUYWObFbyBKLFKJmomrppkxQhGttsICqgGHnQbKPyUeonLMLrqEpPRfIYKwdVbwzOrXScMFPoOTVOUMpvgloVVDmIDChiQhJbDtywqifhZyaYKceGErbVDYwRhHGKygAzrotNpjftLmFnhrxGmlYvAvclNcxkXfhMIiShRVnwwgABowIbSyzQDXTBCSJPYhXOuAiqNgbiXhwsuFNNzvLIkwICJCAYFXwcRlYNNRCCcKxwNNxdZRikJJKuKZYaNaLkvjfhuOxFuTpuKCZTonJHBcpBWfEWfgPdYKWFgAPpZWVPaQcyIbLKpEsneRGnUYhiYdRMXhhzKisiKuncUqHtOaNkcloihNLJIwwUVcnbZEcaVtzYkGbEhFnAvtAtoWUagGfpLeseQHgWhzzFkyvUkrHwBrLOzNHrVxnKiHHfWmBnQYlZGlZXZhXcaaqGRkglIFNLaOktxqUaNJFiqxqAGTeiIQGuLBlbLlhMjaHMPGRbCOaPKJnNLkdDrCmZkDAzieTWtctzpyhBPzzzXDVTsJBjBeWdUAdvPMiZPovNpcbjFozmolpZlTVKCGfuZYLsFaLtFxctaMxJDhfyAvCJATrmdopdQnOGGTFZJPHkzGyoIOMCpXGGFssIkTvkgigjoGcXJIfJwxjeCyiaTgDxmLtlzBNdftsxQxaRLgTqiVqayIiqrFeTnDcQFijDKGVOiTtOMpMDkxFjfeGyczsWfjlWmdyObfuHhsSAexjuveMoKkWKUpivmWOxefFqbsfQnQWmcSvRavDrPzrmxPTJfWfApuOxucbHxXFhOIvRTLEtkndPskHYVtxIqtvmvZAPcgcuyDEEgVFFrkEeoCOpbMYAcswuorvXexUifVxuTQLJIBFIIHnvlpLKLPgFFMYDGDQxPvaWLHiITaOWlbxlgyPhGhOHbJFeGScMEwSNoBHIVCJRmgsFnwLNjExHMLfBPSHDwCfzSdbUgUlMWJTfBuXvPmmASsRmspJoCWqRwqgvdiiSBoPIQupaQbjpMaJqsxISlGfDmjgdueaUnMcNZdGLLZNeuITogPsqSLyWhyEodFecwsTDaKRIsCCoxfAlOgzMKbosvVZXEyKSoxMLxfiDIskPtfnECNzeUpkSiZRBSiqdncylVBqiLoRojvVvwxsbLBKQbGvYsWavQsTqLwsXBeElvMLsptOSVtlGWYIZQdoMVGSLFUsERFUWpTHAjxATsFeSLTknAGNtIlQwPDpEIIrCqIRnqXqhTBNzLsfkHKmmrPJTdrYcaUMwTZyuqMkFMsovPcopIJOJfiSsTBucOEucSHTRixnoBWNoJzjAPSDvbkecnQSbENrgnVZRBgOgWKAtlqXJkfXbIjwBIvPNRxmrCERUXPNzghIPXGhrJneCxxqFTSjiTqEpHZqhmfygLGWFFuGZfnhAhQFnjjuDEJHGZcYYinIZOTQjdCUgJqOXaCMOphkMdvRnnfaxBYwJnFgqyMCFgZOrvQvTEXWLJpqISoLrNFgOypUdxLtgQtNSiIlBGMOCVsBjpyduTppWiDRDqhPFDMPHpvijYfOuqDqGjQDjSkeCVkXDRFeMEGuTdyTuGOymUReSxJVynrVhUhLoOVFHRivHbZmHdPifUyWMVLmsHueFRosJObFhlpKoBFOtXdgIJGBdbNWsgbTFdIlANyRjJHAjtHtkSkQYzRoKoKXqCNoFYJOXfTKtOrhrPuGFwclHdXyuSnoOyFepyYKmbNMzerfgSlVaMChhUuYRGnoIrJvTVmkvawStreuxHmLLqBhvKJsRhZUlZxEKvjwLohkjIHWRonICltFLzzTxtnlWXdVnIDcbGXyQSeRHQFcUhtKcFZgcnvhaWunoYaCjUIpwOaufzEmwuQwysihXomDinFplELCJRQwdWCzHcnykxKOpRZBDymwuRGzfLbahUfaPeYcpVYztpvoYjqwWsDxywCHEusXCjaZRDCDSNjXLrUvYfbFgyayHOQwBezaTgKEtgfWCkjgaDHyWHDLDHORpanBvQERGJnrUlIdPVATxunBvwlRaaqZIYxhuHeYMJFNdJMAcIQsMRYlRsUNunSdIkokAmWOPEMWVseLcCmtuLRqPjsAktdXVVIVNCzzUTbTgCtdlCroYwPomPtPlSiLktRySvnbdFZmsnRsdBSpuUrGMCjFukDNXigKqBbtxVhtysMNyvnSJrxTGprXbogxCdtVeWuVThpsaUaprvVdfHVkeGfaeDMVgFIKyTxunioPLAkLTWFLtveCPEyOMSgdBxQQnRjnfKWeXLmMZvBfflUQkvdEAAWyyUxDVXemRKWHdCzyutmwTyXgJaNQXJejLiNFXiwVQSIEXpNLVrkTrrNfZChVUIJKPTLQtHdjyEPzUTpwASoBpTdlZrfqXsigpYPCejYgwzIiJaGWzMOkdWlompfcLlnDtVzwEeLjgYAcYxkTyDEsKDBeJhlxvizFNUAESGzYPddEFbhYzuZVvVvBzdGWycTXzBfJaWaGEZMWGVWajwyblohxAAmLSlVNRlSsASJeZdopvOtLIgacEZJTZSBaeGyKojtUaLFrVIVBUeyrlXxwgtocbjJaSmdwmYghCBHBEufoKOwyRBMKTvAUQdDndTROGDonydBZGpHBlALRTucboIROZfYJuGhzxbGXfMDazgyZxdNCcPnEspncRrbIWwAqOeWeutwpuxbYSDacCAYFyPzzuJVDhjUfcwXFuZmYenhRqXjNRMRXyhLOjvcHuoExIfRxPLUuxDQCcVQMOPwotMTMhmmjARPSaXfkNQbMmUrkGfcaRFlOKngTfrWPDRCtEWhTLywHoIRqsEVOMIBoULXEMwmgBRNyyeCWrMrGgpMWmnCBDXMOOGSsUiphBiTXuqmRLRiqgTDxemoHLTXWqcfhurUfxbvcRsMAUKEeyIhiXUmjyGhxnDqbgOPAHWozGhORmFVeYhdegKPJugQNenmWlsVhjpoworwtPoZaJvSqHKtPSdwaxSAJPlZxwVwkWvAdyRptLdAYhCkIotZrAcMaVhYsYPVfzgSanYMTRgEpffLtukDOhEytDVCtwYHcHomJVOhMeTbysFgkXozGevEeFfjmKlFceDgBtIJNzBdvKQzSEjMkdYnEQEvYgNYhFHqbTViHlcSfIMTgnXpVxneuQHktZrNRHqfQVAZfkOpDdjPsxfsowEmVakZGQuzJuQWGAxkVFAqcFPBLKVXMNWCCfVfLzkInBuMkPaaeSKFkuIUlmRCmXEgatlIPqOBFBflvJCASqlCYQtegknMfWRlmLBMpANfPFiXenZrzAGURKbRPpBAOriIeEMruTpUHceTzUIvmgGsgaDEaaLfAneGDYzqchPqRcdohQsUFBaxWDNqnpWGNkevMhSHyiOCGJVtDCyzXdhGUKmlQvZZMpsfmkADDOTTLNIOdIGgOmvWpTbgmCheiCAyJFMwJSwcKvpnkDfbKKuTNuujxCksqeFnGyAfmSWqCXUtdwUlJGJimLtODcuTCUQboZXeUndGAwvpWkJIhdvlDBdfqQhFCMflpHyusopoqvnJZuxZcxOrQXSTRHtqRnjWCldKUVOCySXyOaHEfsVxSXVtYdMAhnFfjDbihjATKPzQaeeSqkhtvFkirmKprDMmFyuSdKfiQrGZXNWsjElxqRfPoKxeWKxqSsTCqePUtIKclRFYxXsCzyxcTOsdsamTqWCIQGEPtUbtNKXesEIrKhfopCCIXLvMrdjIYFvTifqfaQRzdbVnSPkNLDZuZJsjbSigUCadEVRqaylKWQZgHXkKgJFMjPfvsQkBUEoPVOMBVjQmsUJqEwHrxjyPVjjJRroZDHTGTmIWUraUSwWJzlXHHtVAuKcPblxTMzBDSdaytOdioJUHnwYeEwxyePktbMhcIumbRRtGxpSvSDzuOdEDGxaIKkwRhPnSWXZYCOTuAtKnPwdymPVIukArjRoYilCbtlHZvECnOBdnTZoHReaoByUxvBhUNOcqvVMobkstThYByDvJjENPIRGhHjCnIeieGwGiTHyCxFnxlLDqpCjUTWSClKaoXwVNqNJlEnRyqZAhyBrmGeZLMKOqJNZEiQXbJchlhxZGVTtwcBQsbIrnXCoLXrKVpDPIUvUqtqcGelWtpddPZRKrKJiLJzzvJZeKlHXebtInMdUWsUdbJlmaUjAbXQvUMiCqyicyWnsRPvfKMUPmlSVbsloapFVURHwDOsBSyCslSgXDvqDpcICoQhlprdXQSidZhwKwVBusMvTdrREZUUIOwpDycWVmoizZFgfVdahkVzsTNkYsKcCSQUovZUCPWuJENAEMJGJwJfEtCUyixKscTTuwchPHQRXHAnrbrvcJlETYZkOcJeuoOZiAKJyzwPnOnDxevGpZiIgLBJImCcTQnpwRyBkrXCsJAhneCcMSEqYmlKnywNpPmIKJAnLJwrnqZxSHVlpJtFIbntlvDsYYNWuXRRnPlxGSCpgYUXSGHHvzuyfoBpQULyMTQVKzWXpYqrwseaNQDLjFVjVDaBHXdUYJIIhYpLRRAJAqHbFmIZAmZDDouJavMxJSNDebjwJVCjbyFSsHEVjRHQdfuUoUZWSNgwRvaMxnkATLTBWMUzvmMEDGSltLKydzBymEaQsVxhAHsUjzUaxGrgVtCisosXXPjVxKmjUoQaJmlAuNgNamQOJYBETFzhcJAboOIqGNDZHnTCcuVBaZEDxIrhXbRioXzEMOTEOUjtEEjmjMVKbkNhLfXKxaiIspXikkgpfJQGlHfNBrqsxWDgBlzvnptPGAxdhFoWAoQqPQfHzGfsuAwfoqGzRZhPstMldVsYuGzpySAraFqrYINGKhlyEziBgtAxzBiTvHplQUrhDmiCDuGjoEtQidCYlkJGVEObQJgDLtCRTHoqeCHlHUMXsMQkozvAnLFdqtVsFnAcuAmglYoiJcBJVCHnealOqqARZsCpOAWtPsHNpgZNppwhRNZOIwuQlTWpVEImwvGKzcbWVrMFVxajQNcmMtrdXTdqgCMvwtkgVpWuGQCwQWKbdzDFonDhyHrUSkSuikjdQqfricOtpHjuMQRfAbONXyjZzhpuVeHVQajRVCZXPRKrTPVWFlWQycBrkZknZdidOTOIjHnBnioRURyeutASZPRcNDaraLQFdrKtRjKbxkddpsGfRdNpFAaQmEPnhNYNwHonMnhOTVjKyUPrXfaXsFolSUBORZmaQlirQZcLnqxBjINSEBmxlDVVLuzILjZjTdUKlOmUEUrIvWnUlfdVGQQJwSkSAazszuYAPvdcuewTVaqkZCHWkjJhjuTNHRNdRBVwXUaVpgpnaFTGnRuVJIQHGNrmvEuxhJVBniJXEQYrONoVvTxRGHjsopEZOZXHhIJpzxFjUyQyqZfzHTcPUQowwLoRsziXYZFpYlrmHDNBvIDyWjzqLZqdkgSRxidrqDIWvBIxzWJmvxDGzMjwsHZyJATTcRHDTjiGbPJyVmzdNtwIOVlabtRxoNyuyKWdNAVhKxGVFTvEcACSjwiBfichuAslrPKxJtaqObSZPcjQjeTNJIIazLQrJYuSyutVvfezOmpPQMPsqgUCZuVQISosJbzNRZzFOTQNqtrXsxRYekZhBCsUFvbRHsSFqdRmjRgSmslacvZXHXdZSjHooRZndAWjQTlnEIcKrJKKXmNdqQzJLmYsiErOpVaJHGWKXCJdUeFydZuYvLRPFFHoiEXIXKVyafItkoqDJcwqQVfZUYSyllkNLLubuViJXYrsGooZiKKieKtLKyWefpamtLnxaWPDdGlMCiXfOimxvKdyBSfgiGcHnwdHyqravheuNRccezMxbcMTbRVpaPAHRpyyMLsrTNvrdvDjiZkjcVircuVSIyBkqbnrwBWPgUHKjOhFmgzDbDcKSdOdqgThtfLjgwSkhOEXYmTAJzrIMIaXDnNxbRyjUCLTBtUbeNEulQBjKTkCEIplkfWeHzGxHssoBFCImNHdKSSmSFHybhqNUTsjBAkfxwPJXfCCfwoFdQOTRJNaghGMdNQihyjvNtkYkgjGcipjiuMDTzjizVwIbAETgSGgbKIFpOFVobATZEKolofjvcGpVecFvSrRMiswjuUPneUqxhJQkzqHHLQBpObOtYFpFLzHohbWPuyYzYRDdKfTECLVnmaXFTAkulmwtVHWWUIBboBbrpQaNwXXPhbeQrOpUYkMHHWnwXLLhChyDHruaoGpQzEAEyfttsgoSOEblZaXldnXCwWJUZsdHeCTFqUqFPqwLzcLXshbkYjNPracnwCNTPZzwskaEfbtujuTMtKdzNJiBYpHGkqeRhaqILbWCxcKiYmOGbNMLGuNTdnqroZmZerPpNzcozbuaSxeGqbNdIdNlRSqgrArmPyRDDCsLPVmvYDqRRhAefiZAeZpiLQZpZMPtTOJtHuZlNlCyzyQQgtdjCRNJcwErJnGgAxvUWmcVkTAySfbKMHHKUFDMKXraCEghrVXRWXAZvBnEfPGweRHfcnKImUapxjkmmxupMqlBpkxDCHjkBuOIGrnNDFXziTVdxntWwKrKpNIKyDPDUwsbiLhzGHICutazOAzqplSdnvwsWJQVLmColqpWhOUnSzBzGUNdIBsKvTEpdutlPzbDcJnOgsdmrVigRPNTXCUVDIaubYFxwHrCLYHlvdPOUCNbTFpCiQBapzNrForSNnxtiRnWPUbSmjBLcrpRTLUgcruTjtdTldmsHzpbRfCGFTAvRUoIgwpyfplBoWpUovZdLZAfTUgjCvSWOnRZYhcbTExywDsuwVVgOxeVkufPZFafXHjTgWEdctdYfDTBKVdeHsfMdXVIQGvDokPbvTpuVbpfZkvJiApsyKmVJMdbQRtiBTpjzmxUbtMnpySmqTcogTqpwPYpbKexkxOwGhRlEKFnlzaTXYaEtSohIhMQdJJPxajjnxmoXlJZeTKbSdXxMdrJKKwOWXLnjeLxxiYEdlOZCbNfYBOIfrpriJyujFqNEmSwuZUPLPjqxAnSUiqybxwWAGSwfoMpWVpnHTYSobrNZiwwZqhwmuraEmbuzWNjzKBXTLxyRcdOrZtCguISFcWSNtkUiGyDpYBWTWxSZKlwqlplkfHmrdJoqxOJrYOzNINHQYVAnktlEOfjiWHUzJBTdHwKVcrXKEiUDFXxjxbXctcdnIWInijJUzrIRpruKvXtBTdPhPqOJXFnjVRgBQtiabXkiDBKUDedERErZnoRdaAYSEEGXKGwIKkikxnrWZyMHkWyteRBKgaXxfsgufnzwPdpeOKEHZKHNmlDXNfiLZWuOepjEaZoHGeFikiAVoJtrkyvAkGpnaEaYVchPMVyDQnRtCvvnuIMJNpomddFpPgCdKZseAiBjfjMKcFjyiWklwJPGdFJDrwjIuhNnvcJCfSjgQpDAjrtRbchpSKlrdBQovJngswUHVzkJfaLZJrKTMNmPYJLJpQBWGANxzkkLuWBTJIktkicYfwFmRwVZETMZbnLlFgiixRTjTOvQJPpufMMfzwnvGhapQnqczMUKHXTInjvxuSFvpZkIRdnDTlduXIcSVDzlecWvnORlUaDavduvXBUMniCJtSxzwdGDcECZYhTmCHioNLYkigvXOngIIKEHfWJSxrcWKiIGENdoMgFYNaBYZbCQWcoJTcYMkNAoHTpuhEyYuLMvNXIomZiRmFoaVxSpgMUKBSuXodcSpYefPqaECOQHojIkfeaLWLLhlWIOPdQkqTPXPcXzfMQgArlSxCgzJCfXeFDMLhNKpDqbRphuglVJeNyadDTzotviBzkNmwOugQZUFlcVJucwJnbfzyXVqCoRGxQzkRLNGLkzBfenbfFQsixgPXuNrGgFopqtSiVBOhZAcsgPZAJfzhlRdeRHNHeslfigxyDsrClSbdBjBegosEwKCSaJXtwsNrBBxuJNuphzMYqcvNkGXvfcdxtrMYLCBZeoASKfGxjTchJFTWjeChEDdXdilOQCVmLjCosZADeKQWWJixOFamOGPfVdCuuTOBYiMuADMNNpJlpsoyOPUYlFHSDAMZsnHtWoXqjFgYGndWweIhdvVDTmgKZvFUHhtqQcchgvlxTUUPrsMULCtlzGyGFbUmVDPbtUNrOqEBzrjWxdtkmJZENeSCLGNhZwWixisymRegOGcwtcoGCtxtihhPajGhlbqTDbqkdsxsCsqOrMDsDyLqCaSMxAxYqzekgMjdRmEWTawYPglCzhfRbEIuKAKQIwhGmOZBGQnpKdMLRciNecohKupBnmreriuCLiIgfPPOIcvTbCRGAtTfYqZpDJWAmZUqXNceKjxVsorbcCdiZCTLqWdtoplBAyLQcGzMyBkkBhckAJhXTXdDQVVhgvySKxMyXQyMiZCJBJDPXKzHkzBrjHPzxfzdIZMMqaFFvBRaZhefrgHVYvAekGzntrVlwrlBtYnJkjvvonCiMMAsrlqVQYSaVMKuESACjJmZxDkfxFnvXSlxIkjNonquOBjKsJhcpOtSwvCcvrAEXRmPGROIfcjyyDdlWrPlYWMlXhwMnWWbkWLbajnsruvDIABvTchWcjasUuTUFMTzxEhezDTLAkHObSfBrTqlbxCmqEBkKBQTctCMoShnhAeFVIpPjGmPyYunGyrONylVStOVDbWxoHDURsrhSDPCePwAyUUPLICRGbSyDaaEqehkKkrzGaOTexvoPqWOSAQLInBWunRZSDCOEcwiaPUveMBOFMeOOurJTghEvWpSvzTONilVBLucwYBinFpTIwTwjergbBWBgDnxBXwjzbRXLhKPYZMPIuOdcxVCHXHpbZKUgXPFzOKmsqZZBuNBwdOaecOFtXrISSFkeNmvhbKCIqVnLhWFEUMwWFJRMyIcHugXcChheaWgwoSPvRBSQmLygqLCOKYSnnQgiXXIUjmOqxlFVVACFTSfKdQRjNUYXDqxyMGuRNsQtQoHONzFahVInMzYMAzCghmFcWEihqSHoqrjuSxODNBfINzYBAcbtOFAHcpvCZtUlLPTizaNwDIbxsOqcWKeLDrFoCtyfKDyAdfDplGiRHJYEWjdZPFtCxEBnNAalaFJcNSRKmpJXPVGzbNIZDPBfXjWdlOXEhOTjdjOpjVwiWtiiWOgNlFwcVWxekfOrSBLudGpoTuOHEcTBOBhOZjrIslVsEqNQWEzKLssDgwDBxbKEzEYmFUesSdXcKIBRrHzVmanmpvmuUtPLlNstMfFqDjUNRZdiZypbVzPwBDhhuYeQWbqSCnjQrXvSgFVPNVQEwBElEeNGhAesPzVomIYEitrtclSDjfVGbVKGQzaBOeWkmthhGnaDnRstFKHpmiFDshRsTfOUgEiiIGSzmAaaIxslCpAWdWmzkmTsfymJzBJENPPMHBZbIiEhqyBjQfxXVAmnneiBobxBnthFeelycdwPmcZnOKescdHpshemLyiBAnRjCddpNkbFXYPRfqGcrXpbhxnHOBthBCjwFlkMBvFDNMzWqfcwtmMsKTDEvnTFVVRELoZhzydvzOxSvincKnvxOsvcxGuHhydyoFQiTaQreDaXpnYFkimzreRvRsjJuxyFxjSJHwQlVLWaCYiBRbOfapARnzKRQjnlXwsxfnTiKEiwAxTKkRZSCoKbovqrnJxHJkuzrGPzDCXTnylAHDFRzwcfNidwVSfKMwmnlCuUAqXbboVDSbFafPMIHVBHMkLfcdivngNPLCsaaMYkKcFkhCLFlYXYqmRCkCnmbVpadHjFZsVNixGdACBiFrSzgGvvkleagFqrijRuAUfBwEaHlVFGFgNALidampTEeLCAJnlTwdWFAqgULRqsPXcampYxVWtddubNZJJjJIdEOASSIhzetjneKtNAjmFgsOSzIpnhGHDmTxaCrkdZyXuTpHaEuFugADzQjUmnejsTIwIIfCKxjsKOWuzWtdyKAYRPbwNcNPRaOCtVoRBAzmajyNyUKpVXsFawNgEHxAkApcHHpJJBuxvOVHFYPyOnnRHnctmsCDRdbQlLqKlSNIAVnZIrWuCKrUEbhWTLhOJxBMydIKsztzDBBfGRdNddTsUUOIkbymbAxfkbgNVyUksCcYTgOcuXHHJWOqRgGnJSLvYBLlHqEHbHqscykbYWcMBxVZqGuliLakZhBprcUBrfzSVIaNCajdjaFCoFpOTUAvewYllYNxaLSvNPUrvrdqEeKhdcMDDXGHvgWJawoQuDvYFZdfsNZONJfEnNEqxdnPAurdhoSDLyKhevREMevijkuKDfAwtxRyxqxcyvMYidyhrFerQvRfVmsSPsahFQGCyQxVZZATHvAMFmpqxMYGqxzNGPnHLcfoaQQBzyHiBDQiLPIQZxMfEaKEnFlVijuriYtjEeJMgclfOURzqVNXifZpUjMzVdwgfoGUfWoWUTKHvVsXvBqjQGSCrEjYDMtHRjRYZXxvcsSLXxLpAJfeTEbrIFHuqCjcZJtNxsSjHElvsHEzPwcjdpmGaKCjukvSUomTZnZunnKUwQeWCWwxxJcQzEbEQMiVycimntgnWsOJmsFQxbCdgipforbalVpUlcbgNjidZGCOnLLIdzDssMDMJHtqPjmPuRbcUXxeSnRiBWAEbybLDObdzeZxbloYmfqTbWyqWwvNJrPCeTNsVFxXaGFcyLtsbpVlfZxZXGHhksfUMPSqSRrHMpThkZVpZeZhWYgPOgpPGOqaTqecBiayDgDLNWjXegROvTJgBaBBuqZmYSsVVCPurZJsPHJqFgLmjbzhJSNwTlZUtnMTafQFLVOOWyJyiLyrFjqhgFiNAEzMBNhqwdbVcjayjAeXOKnIdHIMUqfzILiYfUJXbcaFHIzjOAxIaMAxUgjpZreRbEGfCYlTWKSbsOdoQAesnXEeQqwOqkaroJNVQmbjRVpWhvolbgNhNBfXPIBmoEwZYcBVZrmTDoXRWanXpRkYiKcvahFVVrvYyAhGsVPbrtHSxEIOKttKRzPwdrzUdFsUiopkEvzOvEDZosLScCpgvrlzwZYhdCGTXuxSqTVCoRPuveCavzpoFyXkfibmZAzdOTOSVewUXHrBpUGZpmivJCkdlgHyabhQPATEzJQiuMcFCsZvfojcrqipBOzdYpZspBAANaaecSDdhDKDNhzMUAIeaVDiKbFULXRYsQslGpkszdJnaNJhgCoAdlNuRtbRugHFFdoCjMZvUMWXtnaytOZVfVdQCRvYkCewSvQCbcMuPYPebGhOjIPvFYbDukrboGjXtocIoOiEJgroMbjmhgTdUJFzoGCFNrdmbDBmrujkgjmmmQyMQSJXQsjRSQsEdQlErOadHmCPWpLqQXYKluksyEnjOLxldVqaqQVASBlmgbQcIomQfYEgCqQtaJRGLyXCzEXtbbXlVWJZaMZhrmtnhoJpLoTtQSdvcnnzGYkvVQZeyTatAUvaeKaSFXQEzXaNnrapCaCVOevEJcwgafCBTIYgivLEzBwMbveikzFAEnGPuXHkDFnDlQQDaYYQTxmWPuhFkcPBMLyGTKLUGxGYxEFiPENqWvxVyaZtJcmWhJiBxUgteLmzDOGrHcRCuxBNOEGwjzDAQHASgMgUXhfgFbvfFAnDRlnAYIIJECJmuEVugZequLKkzNrApMXHgNhfvWjKLNokgJtYgbuZltueWCFbcofWOgIzuBEiKlTqUKiKnqDZVApFjFPBvJSefSNoHZZvIDsMfJnzNxTHDutZzQrGBKnqpJHDWIjDhOZBvQdLiVIjNDNASAVqoBHcvdVJkwFQqjAwiLsHCpTpgAFZUuogGRyZwDXTtXSZJYGldlxZjjMjipOaWPBYVvYJHjHHLNSgqlgwEKusHkDyQfgUGKWUfOsRCrGUTcLavfGpGWLeftqxlPmbTbanTLcHFQxSzZuKLIIvPCwqQjMXaHfqMWWdLobfyVbdzVvBlTXdgPWdFuWSmFeroILDLLlcQmRvHsxMazUBXXOJICgMPmfCTagMkeQoJBWyqGzQfVpLLoSAKoPzJyIcRxmtBmQSvbsshVEMXuRGpCCBOIjEcSmhjiBAiNpgWRJdGKRgXmGQlFJSnyiwlGuDWfYYXvdRkSFgMThWBIwMXisptlTaDgAuJkWAXSUhBcnwDBdoTViXxScARhzeoVOIyOAxPqUaMcGJFpbCAnPhdddENouIjLSaZRRzyhqjKMfPhwjQrgDUiOPsKdNabmcTzJqGsyiIxigMsUnivfKCbWMsILauIBqngEIYjAQUYAYHxJDkaFUahWKRDyMUhCEbyMYfCslujDRCIiZQPVRTtDMLExdaaNXBNNUSyXwMhNkoVfRgBVPlVtCPmvFCpoLkCLxrPbOHrEbzwwKwZDuNstygLNXMOWeFvXthVviLqXNLwhvDZyWUiQVayKeeldhRHWWcTVCiRKpoOZEjKxZPoQKtNeYJxHAEPkNCePKbhcWRRgpaYrCocjdCHGbUGNUdukBNewRESackZGXtkLBDgHFMyVbVEnTTgZxjTfkugFjjmcwZrPxzDPVAjzjuVzTuIKhTkgMSbRgtHJquMlzBTSFUInmuKBKqaGfcCkelnahIGkIVnOuEFBuFhgKpgrVgFivKOiSArADQJRLnCMYivdkUzhRcxiTtfiRumVEdoAedjkmBOpoFnEltHtekUMYpVPNSqZXQAhFpuDwYIhaGZyevqgJAuqSUtvpUvRXVxHagwTuhCIGchIuKShoewZylWLDzYYneTnSnKysgwuAkUETVFTbwhPxBKMLWMIgRaSkcSedMksosbEhianeTpWHlBslvVRpfewwlMcKLyuQDOyVtQbMmSEBQAiOEpEplvjPecgMSQJVzQyifCFXtpAABFGKFnYFEqhLTwScfVpcnRCQPcCJUPAvcBarhTNYLSxCfaJmNjqYAjrLGDdQitFFmPDYnOMxKcXDFdAMLcjAEAjgzWRLvspewpsdIcrdygjvqurILebCYrDEjHUQSmLVOZyCMgVnXuXzmULeSpBJOGekiZuyhRgeLXhDYioRHklQLDPLruRfjAbRnYGVNNlalKQIkSQFBOotODMRLQblPSsvdZrMrUgNRWyBPRbToYTtSrVvyFBIdkyxDWqPuYSVcHodCknCpFgapadTdfCIMQDzqGuTZqFiWVgdgFBUYRHuiDHgNheooOioQNajcuHHWEojDrPmkGmtphRcYiOGQbwQuMqOvMbschQPMOEGdQlNHoOZZSSaRUZiIozqcQbjXqEvJmdnPeggHXDolmalTzNbYibpvqnmxZCCaRPjaAhqNHzOksFDPpodHTyTdlvwgXXHeLFGByqTFeydvWZylwbnmIdaQChubEjKkFnAgihHtzwNLpmfyLGKaGQPdjCIbfUUdmPGMvAvPVTMTxxDrrGAcqZXtyvkhSXVhMcEqtiplBCGMogAhzAlSZimXNLTAEoGBlIDmzOXFIfGOKPDlVRGcDyuEpYnRqCubdgxZQjruenFpbmSrWpVTgobpHRDUQShtKsEEaddBRlMBialgWFIUkCnoXMGzUtkipLkUeEvagMoBcuLxyjDnkThMPQDciVAcLGeSdeeCxMIKBNKyKxMnYbpNgYSAHRsCcWEonHZrQINFOUZKzeeXmXzMxhIXvqghrqGFFTcPThMzHioxlaviosPzUgqDvOqUthANTOqWZRtvWfxKmZonbxkptqwVeOYHePmCWGuHzuVngPoVltGiLtYeBIyHETkmKdQajoiwRiAbIMHtQqviPMMIBXUFsdcIDuURQgYlwNHjcLhHiVBmOUnhqqYCHwOyXPuAbGBHDPgeBiWzvnWvzPdDeUUeWRTrBxhuTgptlggNzZvQxjpLNUIzHjpnNxavYTjXvxzdVMNGWvTWLoiqofwIcZPEIOgpRnUDeIzCbTxphgmZdjKVDRlOeCNVivLCncxUjLpieVTBWDWNXNYmmjJcBBcnNvyLtwAfTwBeNdAwWzSYhSsYiNlkiKXLvokchMrIgcpKeabHkEYMsKtZCmmVzANYDWCNXSKmfAFZTaIzmvNpGvWRIAPDadyvUraJrATPpLelXTxLeUEyIZljsIwgeTgEEaHonWkPhHbqpXPyYynrxqvqHsagGVzCBbmJacUKoSDgvEEkFCqrOZlwgvPeiuPXCbizslvxcZowqXNSKzirMyotXziDjgntcCoVyMljwjRlWjhhJeQlBnmLfcLpYNMQDlfEsQNaPggbOljejsYGzMQYyMKawKqtqXGrlupZyARNCFFGCKNorhBVnwLjjkzdEXOzJlSSvjKNDnhcEfBWUNFwfNiCMtdmkpFHbaZDVosLRbchBeUMwYAaKvjZqQdsOxRbfYXBsIWxtoSXvbfbUxEIXdEdTOTnOHUoVnctMOZSAFjWXbUZbeimSpHiSnrtvuPmgAyRuITfyQmmvQYFdgYUFQltFmLwygaCsArXMcidBFpEBpwKtkZFknwBFQybfBNJIunUCwTJEkaENqUpSyHcjUJOIdWZzRYBpCZDcxIHIjdAqztISiHGmrAwnWcLsbRNtkOHopteVtQditsjsyPDxCcHVsvPgVGEforLMXrRtrPLujGvUEimCRcHUYSOGfwtYuOQWZAsMBeNeSvaHSrmIbKnrunHQvjSOgulWgbhlAvnIKmVpRhhFlkyTGWtiVdwTKxkRhRthuaWyHbpRYywabGSImiibogmqDDlPjZPRKkSouqBITjYbtiTZDeGMSwiCPoMrHmbcbyZRVfyGQrLlQEqCTOHhKAAATRDBgduTNWBxqrQUCYzZrMoUtqtMNlGyFhgeWVkMRIyzYfWmoJbWNWsiVjphKxfIdQqjMqCiIjtqPQKMqwbxHdDPjTBZpdWQgCKUKehgGNMdRLIiUDjOpjmZvSyyHaflUbUBKxKGeSHOomgOjqJCcMbuHpUdqfiZzzoHbqyWklWHXihqWEPWaOxUqrDobmoiowGBwzssNoICvRtvUgocZIWfFXBElRZCnYQFyfwVRnlMGqylKjVFZBEiQbopWeZznKGkNyPrEfuPlPcQmySkxAuFSUwGvWkAUJuEVaMGfddlejrrsvNdebcHUizdJRdKESorJRMgiopUXQYdGKzSvKOKwwrpxWTfYXpyqSODbnRgADPproMhHRIKdACmxPbmEURnTkBeXYKYNzspRwiSuWLjrDklueWYzGJkKUUGWBrfusBlSonUpozkNroVDzjZsgNbIoVEWrtQIrkDxjaObJStebhxvLKffHNaCQNUpOZxqziBlcujOKJlkOTlEcdXmcOyPdeogBApNRbnXgWOuyTNIifQVvCVbnepHcXjDDWgDwFtqPtXgZpBxqyiYJSKHuRjogxZdZUeIDiWgBgYiGVVIarZUcInwFaYDwhElqSNuUaKMBsrqLSbrQfFnzQoRbEqaeNwGvzKyscfHTobMVinEzdJHORfcjYFNRLrXXbciTyJwsIiZRfGEQCSGXwANDGicEfQBnuQmiPAcknAetNpLYfemGdYciRHowgdRgYAiIlDynEgwgRODaSnlVepUsTGBMTQSKaDlRssvbjUkHecFrmOmnKOWSyDlexuVAzxoVusasgWaehAKGebWIMtAYnbvovxSJliOXckZdQVVJXgqNsmLXKIDuymvnuierAvnVFkauIzWqqltbgYKqCwfDnLdPWWGIqjepPhvtmrqUKnoWlUqqsfvdzFiAcnWBvEfJgTxPRcKDFIkZTjcqPulNWOgZMWKkViwZFHYkAkNEqhlidLYyoPuenyGwaNfSqSkSHIZzQZIsTVukcvRtRPnPcoNiwMvKWCyYBzBYqRMouGUhfChitvQbHAyrKTkIAzLZerdYoAzWyMbrYOJzYUNiNoLhJFEuNrMaqANiMJeCJBnqBUWhSNVfkOEccxbeDECTThJmTMCvlYrxVCekBCcBBJclZcQqSfawMOwlmxJIGriYQkvyyiCJfJSIhhDPzffDHagODuwMhNOlzCoGrSbYNXHyyTFjXsPGvyGrIxjvBCNURAxUIfkwuDCmqqzwhbQDCVppgezPpzUcrzxSUjRADbqUqFeGaNmVDcfxBcSEaQGTcaoCsfMaBqcbEiffJxEvWZogHQMEgyCvSRIeoUAyeITsiYaDdowzDPMzASNkfiXhLQzPplmJRhJeiacNkAfeXAJCPMcDoWVJPQEDqFfqoWRUqjUOLrlpseiAjeDAhxFHUtgtSocOZRWTsgCMsFShNuRYTDDZHnjfGRRLcaILoDaFUJbAZbItLARXgZLPMRljWXHBKrfLovJOUdtBwbVreMWoIPIuPZcSinnsWCIvUguGjqmvgdPBOJgwkosjNKpTluiyNXenxueRenXYXXiOmNRAtmXAFtdqqauwYnEmVqNqnGcqPqoEVTUJyIXBXyEEQoQblXQdITNKhUnFZUouwWAeDKBYtdxXDWsjZUCXJsqCeBvWijPCKhdTcumMLGPmlBKuXocaHAjPwTfzGTxSmlQbYboVszlfTaXBoWNBCfkZnxTYkWzZESJjhqQFOAGwQZNpZoHdcFKwRXZPCdgvvTWexWtipbLAjcoFrnslvNRlzgAIbIpwnHQYFGQbFNzromnsrdzysvxtuwqpaRCftlWQGmXjTAtpRbijjnFmfYUPpOqegfEBYaFvUMDqgpBGTUGnwqKOxIXBuftRORMsOEHcCOXVjOINPqTJeSyWkIpHAUETiAhpupaujpiAYswLACSUdAubUOkjTudEyCNlOwiislQYddbauWwXWbGtklCRWHSsCOTdUilIyNReQcQwmswGNuSgoVkZzjzxmYRQRafTIbTlWDbclnkkFZtJXERrlpztcpGvYixAfJatXWjwULZyZpoAExdpnVosfFilaSyBzTBlkhoVmbpYrxfKlLgfPuGuhPPmnpQiCftDiFUZdEAMqsbqBeyzBwKXtQOVbaMtovIroZhGBuvuRDVwAomrxVhShIpQJyUuvtMwOTjJKOiCEKZsIaLRaIoxetEZBLMyrIUuSFAYfrBWgzlJDnWvzAoYYGkHFvGiSHbStUjzSpguJirMklTfygJpHtrzHFAFljGNAAogKhWwgCYlpbgAaIRyhFrIcegzAzurGVwmsmdMJpkacgZuvMQfGUHmARuvQjljFNDXavpWebTrDiVqMxHsMkCykcWQbbXCgwqOVBVDwBtywXYZUvpSBzVAMRlLqUFwwYFGCneMucTZlfcGUidDcrGTOtoJcSxFzbsctBelezTJpKiGLiXHAhEpdkBEtXjCAIvIMuCjhhquAqAfXVHLZjOmdSfKlVVTixJDFtyTcBhgZDxVkfdNyATDObolKByVjrrdFiaPADeyBUDAOBkLRpMfDwNFhfgtSSKeSOaqWTAAfXzhcPSveEJbFrXvJPvWzbnMstbtYcUwnfpAOUgZFmMFWcIyhPEeoHKnSkduVSHvyiouSwbriiAJpDWlVmDAZDnpGcuhacRiLgehLhrpWlPTiDXAPSRMWKsWavsIxpUMkuPIhrsXGRWJbzbLkjnJmDVeRhStimGtgGQlFDzltcFpCcVUCIipqhWXoAUbGqouNmTXtREmNfAsVIQyxzTziZiBqlSuBdBOJxTQlErZwxtfsuJvFnWAJelcjzILnzCyFhPVdjYWSiFlklzocqCngEOXmmVtgNRHTjNuVamltMKwjKnEbFXJZzCzeSUuNqENgSWoJPYiHOaIYScFmaxgJFVGqAwsAyijlJuvrcGBSdultKqwXrHqHXmeTIQEapjBoMNtpusdHZOChzlyeEJKzxOkWlNVcfHnyjGjOhdBTqanQKzFQaGTLFkQQyaHRxRPMWvZqdRVfexmBttytbxVSlifduYFlYqFlXYxpPrbuDSJVpKHbhWdusQvFAjeEkISigYTYEUdRHDXAsUgBUPButHPuWhYesdWSmsJGJTdtHyvSEhmuWULDMmEMDlddbtNJqdWGKKCgtpDUnOxxdyfJoTJHYifUApmbTteXMYsFvDFsdbpFnAVhnpxdceWwoWAEWAHOQrWxOUfjvLMMoiUUnKsVQpFHXvIHPZgsemoDgBjyTtgyHnPsUGWSPJmODiTLMEGWrmHaZhtJpOiZcOpXhZalMhclbzctjlIPhQjBysUTVUvKzOKibRgDBsESWMSWsUlpmIxObMSmTnJjFkOVXXrVdPrQhkGoajrHaQUmOmSfyGEDOBBzDvJnBMbMSHROIvVzPYoJxGuhftnzRVqmKlLBmJevYdjcrgKlJEFsQUaBKMHORonRYJYnsgMrCiEsXYLhpOaxwQkiExOfETpPPNlVNIsCKHLTpkLioJMbUCHUoUuPnruZdDHjolgTqTCHSNafomdYihuWSViZfXQkACzubViRtAXCzjzxtzVUXdBaTsAGaHfoMsRPlvNxIgboAmrpMKOEzvferGApkeBvisBADHyJtxqUYQOMbUAZNFgpIqiHAqfYkGcBUdtPSgXcddwgkkkWkFxLUQmrTAhVcCbmHSQCGtxmEdEDZGVHUuKJSVkQTamxQPqDyDsWrTBNMppoMLrEspsfzvniNqRJoZIBiQQrDyTOncFywUdDUNdvysvwpdGGiXfVVdxtbSEhJkNhUCdsmTAJRbAEbbOnJIffZzwpPoUgDbPGTTlYcAIFtqOvpzpVdJPBNqtawrANRSXSRSlNgGIftABuZpKlBysGrydyPqbLbDxcedHHsXmdYSaMZhKAejTVuMcoMCbJkgkPzSkEhNpWPEUlOuemzAhYcsMBHqJiToOwiCxwNSloXdVYhDZLuCZCmSQaevcvumiMKdbWFvBqyjWNggBRPAqdrpZmdiOEKLKsnObvhLKPyGfNonGnqoFyKZBEZcwEmsmSeRFOvUcRyvWfNfxUbZJIsqKjZKqceEHgNSQISmzNmOHEANeSqsJytLTdTkwLknntMgtVaFhyTkIcddKtmsmYgnHcjJanLgbaMnWLbxoNCsRFcsWJfVDDCthuMjcTJqbixQGKtkiIGEmROCvNVyecCSzyaocsrMyrtllLmIvUUfKEdbVMKzoVYpllaDyXogInaMrjhSdPGgLjZiRAYmjtPgyrWynogrflFXWHsdbfNRfYsroDkXzuHUPgdNgQEpUPopfQqmntoGshDsoMmTWMdCiszuqSqeVZaHXCLJpyfRCcsAianFfGnMgZQCaKwJocDyQzZKCfxzlAQzvbXYRkPEofGfYVgBshtExZgkilxATQMnLfDiIubrnnPnvUFZCDcjULxIqaFvYuAJqvlXuUFlQkLJqpMfiKShrBpcEvevAveZDfgbejSxbhvaWwagQScdgvDMOTyPBnmyhcsDNqRQKvEXQBDXEvqnhcTHGNvNFxleFXJfYllcYzWtsgdnHBuYuofQGhepwSwKsFeuUEXcZEbiSAEJlAVbQiHWBQrPPOIEXQGCACctQNsjixnhpjaAlqnVjMiBZlezeeCvZfNinpcKQYpBpkxDgDdkWttRTNbLcIQsvzLxtoBPtKTArNDwLCiuHEZtqIdNdWVlJPrsjgOfOrbThdhnJwyqQTxcEIsTWbQwAqbymcACQHzoDzPTynIXiVCHIlGyTdKMItdaFSmnIWQkKjjiCriJnoqlHYxiHgBKcvYTvGtIeufHKSMhkRPmygpjjJfizfHArWQcqCpkUdPDNsfqreLyvZxEnRbZPlXSxOcxucstleBFsWkomtCiQtdzkapvZEAbgeYQsEbBnoRSnOKygNHWxHBcyCriZrbLDXlyBXeRJnzUgKuLQQaltcxsZEmEBczZDulFDMftYxRkeahDizdkULHEtLVBqlWKhgKTswbZwOuKtHsDZCKvVlmBHiRnmzyxAVWVEKsSMVYIJeLhHXGXchUeZnnkLglPQTfUYlrwzGXfMcMnpsdmJhtggZHGIqPTakvVhKOHOUDLkQpJnSioRgTyHoxFHuQbkpXBHJiUXEyWcLOeSJpvUeIphqotSGvUEAqfBaWILYvrWGgCSQCmzuknmiEbGQVAEghspwkSvZXNBOkDDKOTOkFbXqdMPJOWoMviVwVvzvRNigUgEeuYXQzAPcxLXuHYXrGoNSeHiDxgvuzGksWiZynJRxFhrJuLJaYNOWUCtepiLYJaHhePoppfugbolfzCPxupimLzMAsMklBVTUYipOvRHfXGFvbjMWDlxpPfbnVlpiWcoCTPhNyitdOJODRuIUGopJsMjLmLydjDVKTeZTcKnnBdtDtesvzMBdMTYnThluICpJVmcfmXymiDqLThHXklEDXvnCkTwcxtUyTAmAuanPhtQKBNyzMwhHPUkOmEHvZSMIaYULeKaNbnFsoAqsFCUnDBKUzuWTpkkrGmQEGxLyVQEAxELttMpoeFgcKEkRnjRgxZCPVGSTFrgTrorpJMzlxEpKQSJWifkvpTKLQAVEwHMZLBdXUzrvOBDLxBfMRhyPjaRQjWeRZOxZjZfZwqscThqvNkjHBmhiLYeAUyLRLfUornTsTleZdakPDTJODoahTWEAmGDkzIwejHyAPJCXvNvjgWAxfQFjysRjgLNEWAqQYdMWroEgbqGJmSPKDYeVkTyHJAWCBYQXoJPqTxXVhHoWZpiONWtwshWJkPWVIWQvZvemARnYTZhewlvVFKETFIwhkWaLNWiFohZaCJITlbZWpmqKjAEjFFQgfimzjhOKrUlLotcXnXhgkmRzntbhdbALOndeMKPRNyrkaRHwfweNFYGHzoVBDNJTzkLyTsrTsaVMTKSPgovHdkehQjfLmxeascjmgsSVslflYcGXtxiAAxvJoUlsJNlzIlDbpqoTSHPSDltLUdymksbDdLMOFUQzgeRkUgaYIniLkgNMkZpqkLUGqdrbYrFONsmndtWkpOtJJsVeawyetXdBXSULJIJuvCiuThJBCCNulxOzJUDbjXMVNkUXrzlDVXiKdiywzXfBQzBWGQbginVZCVrWdgAMLdtRhWzJYuurKfoWYqLWKBUWsnMXBDRoeHwsihMQJcPvnZJBjyFVkgJfexPwegjRCxUzTugorOobWTWlMHtnWnacPoMomVnMjrUmmCPaUIFOkWstSWFIxvyPEXqBouuGOQdrqbsWIpGMVGpogiRTtkwPVSQFRuJaQCJicOUnCLYHFAstuRiBrjLEmgYoFyJfxTDVIbCsDKAsVhNyaQjLjeMsdfuTLYXklmQOiMUeQVABkYPtOnGkRWWmpIRPWSGHOeSfRYpyeUYpCGFXdsqtqhgKDdXROFSCdBGHIcOhPVGWrVszCCHVqMejAZQgrGbnvnIwIDkcyzuvMGImMjNFlKcKQpYCNwSLKZTVFyHlnaPmPZkoYnfvzpUMQiZrnUjHegUviakwMzisBsbFcFlShoXVCfMQmyGEsQeEXVzhVJZuIttmVyPmJwkiMfcTmPTKsfOdhLATtzgfKXPpmrOtmZfRWhQQwekQJvkEeAMbONOoEWNDxpENBKBzBItDFWjpdCNvDlqesDMotVRkklwPeMCETeSDSgSRWuempFlVUZIrafjtAvrGZuVyvPfwLbiWsCkRFLvkvksuZWlHCplRLurliKjkHTOTnfNBZguMROvsJKpLtFbyJIOvEWMrTXKQtQYLHPKMSeQOSXXdcKayhFfESZiKAVzirJAeEndNUvnzewpzHXKBIThkMuStSJUHXShBGwXeXTrXVteceAtqqufYqifHvCbchOCuzOIsgKvvRLSoqcmesPmbPjyYJtVpHNsvWiwqCjHAbDuLJBGInUgMMAuNcXYnsktvFSwDrfybrbuPunAoFJestxObSwfLiMTyOAWeIlMWflEOcEerEKCHqDuzAkkgUOFlCRJtQkwvmRWhxnnMPfNCaYNGGodXmmluvrEqPdkNLtKdhGbdAyDLOMuhVKOrxgXXjJcIYqASGBSnemeWcXsYKkecXVkhvYzglUZcynfQIGXrewVikEoCubuKSnPdqjfLydqWwksXxlDzuEFhaXaCrolGEGXdgDMMDzZtWryTASuFSBkMyAwWLHUlBgUNqhGHgrkBWEgGMFDwREustOQCJhAQEOJiQdgtzktnIJSbicsjrOFPeJcTzqfTyTSmeAHGrzihMHOiVbTaScJPTclHbxaimaZtODFwwvuarZTKuEOGhXDZGCjqLszdklcjcfoCnDWLuAGlRzADLzbrSUGyAwpRkqQfjFioUcqlKZOeLqJUwzKUOdgRifaUAocnmqGTgglTANnqllCiiADmvFNKRsJiHOswYtyZYSzGEWvLzXbNEgBCAMjfpghRzhBeAPjkfSkpjeYRpMmdddjHWEgdpwGsoLrmYkzOKLJqQFWXxIrtrFreELVJCIwBDQwgbkXcpBLGXriYyXdDTPxmwLkfklyazNkXfVbEHFGUBBfrmpDsvZsiAKRwVMUrCcPjXzqYNsQodqCMORiCOYWGFzTHuHarfRuYlURdSgOPXCxvqWwBcQggppJYDtNswzMMYnuqVJAhHbBPTsjwBvgrtJulJdevReKSlSHYqfZSwlGwWBkwqdbtaBkbkibQeCCNHQDSskGeFGByxLMrhMsDnKPrAwllhnjsUuVrjXKKMKFgpMsFiEmjdAzLsWvmnUkxlOjGRUkFvrEOHcMoyvabzAJplZyvbNUtPXicxFlWhmopnUUeClYWAPBNdzLqrEluxaKUZBtTepERqzivXpCrCevtrtXYEaMZCQCFqEoeohUBGGYqlZKYUGtKRVIXrLwkywgKIydFJKCHmGArSvlnVVBzSVQcZgIaqmRaQIWetfSCjKyURrNDezILJPXQmRLhlhusiaikZoKOINyCJhJFeolPTdqFeJxAmIMIZAVBTlFsilToBGKDuShEHQsfGwudGsMrgdhyrGwfxSOuIrIaHTpaCWVlcIxTAzXStXsxlNeEAGQYNLYqtssZzwRUPwclfYAnSAdpCQGGogGtjweybzeNtAGGjMREryxTLucNbXjymNNpTNAvXeJAlvPOxLtEyoDtkyLdTaUXYWrQZcBaPXtumaPBdwZcWaampTZyzJKakQpBdrhQgcFJGADyXvyGJlRTtmweUTnuiqKdczAnHpqFkLlHDMLFUFUgMkYKtofANadyMGAQiCXcxMFxZXyWHfRpTzBVMopkmsQyztMtzEyYzAMxXKCRatKNLcbvIQfIfMxTUILJzMJbkriGhFmHtmxQrfgHaoESIFjUCNVphhoiyFvngbDrYrMsdwLwDIPTDQMtxQDcJZuynKxGZvADrTmVmlflkJfvyYBygUlRuixxKyTywztPLUyQePmPSodNmlYvWbOOyohCBfxNewmYMZaZJmLfjFuPJCBmLEeYvHxpMSkHtyTtIOTZsIMPIwGzpnOABFfBDsOlebAgMEDzyCwmbSuqbhOMmjLbyosSVsTCTeZUHGljgtozsWOOMHDyrOzQPVNGMGVlOxZWwrCEaVGnUloBXMonNJulhNLFsFKPUfvRFJzIEWmPqwqyDXamIkhUYJwPNOwTfPojtqIWwlDNwfryizZSQdOQsGIlFpYifYtmcwMbKBOvQUfzVdFkmMSQaWxBLsEaSIVpjgbzBADFOCjUXPDAqGvcxIrTGqmqJmcgLKusGDKCMnuDpXTmynMfAuFTKpTqMzkDoqMtRkihVltEEYyVgvVpmqAIMwGiQNJOAEuKQyBEpOiRPbHJwhywbFGZbxsITifguXaPrMYEkzzboeSwZNycGHNsYSpmmgBcvYJwnaTUdkzcndjxAllVscpgHOdqdjunIOcTDsgINoCYpVruRxcgMJLYzALmSyfpRhSNbgykopGKGWOmoyCfefTUCbspYJUItfqXbHglejWyGxmAxncrNQnhkWvoxesHcBzbEELBzKYDzHRxQvfIKARpiMDLibZgmqfhLqbHuYCxRCJXNnrDbNcyqUNgedFawoCRfmmCBvWgAFWxRIcSvUYawQtYXjfPcqkopNmhhomWPIJUnswBCGCPTdbEVcSyhKCHKRgfgrlxMmcvJiJwCkYDetoHzehgHkgreARftOLZbJEEHGnTUwcUMdLHUgYCcgeJWNlXfSEovXCPBiTgyVsqnCjpLmEmJrUbOZiVjjGWuPTRbZjLoMsFudFmbBsGYuRcHHtsTskoOMqNsuXxBpMbhgSTkpOwecgfHdSPIYHOXUeczimEYdqBRQHpsOjHzlvpUBgRIIIbdhLjPNYeATaJLczGRFvmfZwxDONsihojcinHsFUTGkfNYbFClAyYuxbGdcfwmRfhxBvKKYNbpfbVyUiqEoCHqfkvXthxZAkTvDdascPaCHwqqVkocnyOQWQuCAojvuSlnbXCzDmgRgjxyNutStJnpKZAjPVtpYpgRZzNNRwWNKryYaQckpOGVyVAaDOtrbDAlXSUMRzbWZcgSxIcsswgxEXfsjythQdQVBBCjXAdOGwpmwUHGPUolrHrPfqjqgJSClNQfdgzzDbTtMQmSPhhRFZOCMTJIDMioZbOIJNHjMEBTMmKuNZfLgpNlDSkWTlDAsvPibYswxFwMaTGqSgXQgNIMpAUEAVuNwrSCvwaEydDPDTTkTauALMDfQTonlgDSyutZQwIQEUrbfLCwnhkSvBTDBpbAnirlGjOrFuxLqSTsrwSdupmHHumZaFhVyjkOzlxuLrETWAXcyAtXcdrfcPZlTafOvUeRenTxEVcyYBZVUBzqigggRRiTYVRQdssUxrJAFHuGqvOPFZRPfeGfNUozCjhdsfulEeFVRVvUrGoPTlwLmzeApjMoStaVdTjpuPPhRhimFtFRHipneDbanBfYebHBNAcDbsBfPLgXJgeYpUwQnfJxNRAeDwuKKOzwnJWYhYbPeCTYrrOmEzKdUObtPJiJSoXoXzKvhGliStpBgWiHvfEhyvWoLiJFssyRzMBaoStqducoGTMvgejzaQqwwWXpWtGuqjhTdvcrWXwoQXrUTbKMYfHTcHqvcPFmCypoxRpGqJtIYERtSTxGdhSItKeIOzQbPzinnSXbxzHnQZBhbyzzwXdwzNbjlAyCUbbhwJpCDKBzhtMaUfMfgDXExlHCUXiKKwuoWrtVuigNpkTwXXCwKlrIsRhKdScznZSyffihLiKHjoaBgflzmfecNAZLxlYHFiOritHZtOWAOkiKpEARjxYaMbSMglDLzDQjSeQJtToXMpvFjtiHJrbyobFxFWGAYknvIEmfKSFUNZXRYtfNYshGnKVKioBIFrKHPKUpebjRjratFBWNIBAgvnCqFBuOOLeQPSqRPwjnQAscBADwUzyAmMmfqbLyhsElmuuqFXUTVhkVdMIiEEWvPzjUTlOFokNmefaHPeKECwWxlciZvDejfDrXYPetcNdksvVBgzYRyScoMfNdzWsKXHEJtCbRZGplXYXCfaorlHAanBXdwgnFCVQaKnZfrdGKULdBraJmSZboaRKiJYbGkTFuokOgAWjXPiUDXZPwDYYXOtwQcyjHFyMIibXYDbffFchaPfsGlLodtFTKXyrGhxfuJBGYpLiuDCALlHvKhiDCNOHzGUTiVGoapUtsKCaLuuJnRTLpULPyzjVRybVVSSUNdyyQFVLhkXxYhZUbImWkMGwBIkkimWwxpXNHKcBXQZREzRCAwfndsXQMuoUAnwZemZYJVKlSLFDHWmrdrMstscvByAGhssClwZVzVGQgIhKXBaezCJUJraAsberktHYByjcTvKCTDRFFZVxeJEYRgMCrsWajXWoYhCTAVfnoAKtLpKvHgjmbLgLdtYUVdeTTuWAduBeJxXpanFcXhbsXMAFNkfElhlFkbiCMTnbKgXFGMkRdSUZRgtmLIIZHpPQrfjepuNIFhmLZbtkZvWhLciGtPiBmgstCEQMnYjzcVeCRDMcEuAZPPFKzdscmBZJZfcacfjDHYuxDuXfiBcNDCFexAXOXArYDYkXDscDElfCGYSvwPwZYKiMmqonXkhTpoRsdcFRHeuibtYuQRlrSFMvLGnvPRTgKZdgEnKJotOOHWKHksNtDqmFJepjEelJUbyWvCoAYlkRZlacZQUeIPCmPxiVJSSOWbYoGvZdOyARCZCFcPAJGfvZhqWBjpEDwlMNRksuqubWWIdLkOaWhexTkYeKnciOOBmIzHPrsVadpdqhSQWYPfCXcopPOAhqnmGERrEIWxvwvRkogkbfyGnpgaoHpMxLgarvuNeNEPXvmnBxGmantDjegmfQWEVNeMIGAGqTzrAzNfzStbgjdkdsCxCGPRPIzfwXdPtNgNqUeDxOXsNNDhZHrzzPLgSmhzCesYHDAmtwwvZCagHMBZbKzYBcvkkTEuzoBIAEcBIFqjpypWkitpndJoYuiEoxEILrpSBkvMcuCFzrHWbQRHJDmeWllkLYcpEZLnteLwtThICLikhAAfWTwRUmKksDflCvZsWDNHSVLWYfCudtWjmNFewRaxDFfYdVLpHvyxkLxxfIuCQhVqPcIjKRiFWElPirumuVfBYreZulogfhKdyXZawtocFwfATjMtBCIIqVwECPpVrwqJKBHoMeaJUlQOfCLtamJvmQZeIwywFCqnVOWXNSnILfPdSLwhfhLhQhjqHlnxNjraHGNEgFKDAsKxsjswHqFZWKDbUuTdcTYeXbWDkxengCxfqNdWLEbqCmNmqfLGcmCAwvlVvYfpzjItJMpCtdlQinTrHTpzSJFwKnKlZMcCoknHmjFxgEbexfewngBqLwzshrArkKSglnlWiMWJliUwXSMjsItFbeHjiwOtAFQqGdZKNSdgHeEqskYHIjMYOMWhRzyAirnvGyQOqGiQLLyZsoIkUyXlPDcWTDGOkjZYKuDVoCnKJNxpIZErPZXyNbIDzuuaFtQNwETvxkyxtotmNJrzuugrpdDVPjsyVZtYjZRbPVjWHVjNTnPPDBkNmkwkaKiUXcZmRYLfZJIQGmJPYFxqcZHcTRQqjQgsGILXlatFcNvKOMaYvghDxspotwtKbmAiBVaFoCTbGkmjGaGiZSVQTAIbszqvxgwEKZCgIDgvNZAEGwETajfAtztrwjcIBUentXngNBHiyJePJwEnUGaBiqHikGaHsrHxnmrtOnQiqREdLlumjjuGRUXCHtnyntaITFfnUafCoTsOqRuiIyzNiLazYtmaILShGIyLAJhkdNUDtvFrTkEvCwqQYtPYVledizCGXltvgVLdadRltZNTnLBfFzxmNPYhCXXnZnMNWvDrkYmScrugphsziYkhCNNFExXxuFZTXbgVFUCIqtwVYxqwfFEjvqqPqalECoWHNLJZDoiKzukHgzTMquUZqGwTKGSsrBvUymQTvYyBBJKJYFTOgHktXWUZuGLxkHwGyxiuJVbIZawJAscmiCsEqoaePXZeyuSboESdBKHaljftxRTkpKUOXGRlljBBYtPxfMvbEivJtwuBDfhpJHTmxiaToIPQlztGGMlegVXviYvjsUOrxLrJazPukZksHqFMDdElwdJmiEqASjeURjZfDjIiWFiwCyTnsSMgAZzCknfONqsZnbcNWIloxGhzNoDkrlQKZQMHmFUGdKKoakPhTRnGyJaUoUdmemupZWWwrwrCpdeQjHAewqSHGYoltdorqsBTqcWshBWaLEujTwYUDSUYIydFhjKlrbyXgqAIuhJrwrXpDjahvSAyaYPpWjSvSzbdrjEDkhRBrfWnTPRuCagCApwQAwTdkedWMETaZvUKTFpyvdjLpaGHfcekKqRjPUebBTlIthlsImzCPjNkmprzNEGbwcALAIANIRFBWQKWuNhZxEaoZaXIIhfXtfaKllNughDwjXSKiylYOydbrdGkEDGSwyxecwpObwbRUZxNcvTTBAeBilMtLAHExlLalksWWbdHRlICxrcpfzQwnJmJtnOgYiEBwXMJkmXqtXZDGwSNglksUmDmaCAwpsuhWPUZtiKSaEhAEfpFkKNqKZPFEwluyAPJMAsRRhpWvHaUPORErJXMWvpJJtoPhFZmPoRhXScokduxOYVGIFxtTKypjisZQexIQXMVVTFiBxPHSGdhpVgqZlXLRiCQBkNrgdeJJmgPiIxjBTuNjCFwriUhjOiNXQqpdbCFJeaZpLfUdfrugLZjeDYQRAwRujKzxOzItmqRskWforRNJSFQtYZCdwRSCJNofqhjjRuaISPSoeWKJCAKEvrzzaUsCsNKIIAQhBhGkQqLFmQwMnKUoXojgfFnWKIYnGYNVVdcBgmjNtyowDwHIeIxRsgoxVnzoOvjzLrawqlPfOJossQyWLjtMPsvFgetWkgUWBuIrAqmDHOQQJmcIjJefDcrbFYTDAuDFLMbBTuBxJJZwZYYItHuJjxjVDAzYXlsXjinqqxtKWIzvYzUgLmWiQYKYpquVHRYtiqJVjdLJKMNolaCVsvUcSiMwVDMhdeCeQLcYhTjuGOROusYQOvZZluNEbgynKSkftPblJbvVJSgCwUHRzEauVgChpQAYetcblQxFPeJEMHRnVqyYluwbSCyHrryBGPUumAKggMIpcTHoUgEDrwixnJuAsbQnCuhBTfMzWHVtHDRtEBqdGXrudLaDBSIXtMKRFrFkCpPJsneMfkJblWDNrZLbBYqyGjxhBLwdhJHDaTxGtPNKWPzkEovQnycPMhaLyXWRYRgHNYUaDXACzWWTJZPPxPXzEbSQDVETJAlvBwfEkbCbYUwEeQUeTFMFAuwNsziQXRRvpkZuoXOCeKKQtAPcIhugaNYobDNlCcOFFdiRDmmMkUejhhtClWKuwyAaawtfNNQpdRwnUDNCbVNCgmnliqwJSXbUablZMlcKRnCcIscdOmqdgxqTMXGskeKXNBGvywhIeSCIyNWYLGSqzhtLsAZYxLRVeJDNZAENxPKTFigFBaxuRRHnjIdinraZRXPugbtbWaevNzETUSPcgshcKhgvJpUszrPPFSaeZEpRwHqCyTcepmdcJivIYxevejojuEGboLKpmKYkbYSUZEonOjcnEXaFNmaLsdvqfZKlpeZwNleRfVIdIpnHWCLBQYXUfRXiKlwaxwwOECbaLKTgkkznWdGGAoZQcneGCysBrGsgozvnmOlQdZciEj</t>
+    <t>ov</t>
+  </si>
+  <si>
+    <t>KM</t>
+  </si>
+  <si>
+    <t>lX</t>
+  </si>
+  <si>
+    <t>sq</t>
+  </si>
+  <si>
+    <t>qBUanybZqtYnAJBFqsrHSXHhCgOWScjoIqscayTFUUAlqviKUmicfcqRzcNDumGNwgSbKMftnxVorLFmDDuYxOejSkHClCjuKzIQdtedHAZxYKhqM</t>
+  </si>
+  <si>
+    <t>AUQilRYtkRSEFjudCrqyDnmLwVqPVkTFwoKfKWqQcirgEZjOZABUMytvshulGPgIKwAIgGpVTFTvLFjKGxhnVlrsUJrYBYThjIIsvUNbbESOhHbDrILgIcGBHsMATkbcsh</t>
+  </si>
+  <si>
+    <t>YAQOCRxQEuavqslFtNaGaQcxSPZOxzDhnT</t>
+  </si>
+  <si>
+    <t>vEvXyKJwCWrBjFKHWrPnnCzPYjygEbklRozGtdKSnmbqUJO</t>
+  </si>
+  <si>
+    <t>ftvcFejViFNseBJPlVnwuyoiomKinLTGFBNgxqrAxdiqCSphfJhhNErfNoZvttMygxsbQxMEwtVFamusZqJWPQaqovboZwqbIbcOUvSoRfndbytaUdSGHzFzGhqqhHADYDCGQOCvIVlUTFDASjwodDFVopOdjwbxIKCSLwieUgFJsfBeLYGhlJWDDOGaANALwSIJZOCLzOYOKnjwmIqlCVuItUESbrSHLdmOVIBBZsvYfPksMtyMjxDxVJpKtNwCKfNVDaBzAxYrrcXayOXrDVIypacbQooLpprNWMpaEYHPGQjqCPEKSSmTcHrdKShpODuYGUhwiLPOGwWgRACYBMbPpjbuXNnFCIhMLyQkKubquLPuIpkFoVkmWakmSmwRNDjzTRjWBOrQzDDgEwBSqWOkDcBjvMGfHAjUZaGTctyfCpaqvCQDefjWrFJmpuRkpkNKLCWIDUyYxkaYGqCwsEfVxlWbpDWHOMjsfnXelCJUHTgVJQtPRBocQqAqTVvrALLyLTcLrJWTrAHZPhjqjxYsWLJZSUfCNYErxlGrzeBJROpXGDlaPElfLkOmmBwOLzeRhoLwTqirgVDPBPITQhlifpnBGXOZiZOOJZTMVksMnWMQWrInZvmqZotmcASYHaAQzhrlPCvnsWHadNhbtgMoZCAPzNkVeounzeaFMwXcnuNZAWyDCFstlUCmoghKlipirldXHPJVeUylKsZRJIBONilNGsHJluTDczOeDEtfoErcluQCfxfYkWNlcovdUzSYUJLoTGhfGXCUdHiBZaYNYPIjAEMePiQUvNhHKAXYeYZkRjYIBGhegPAhGpUQWayYGfzLatJkwGvkKQFnWFyxkgRbTjWvoQkFbvIOMJqbSpLrQMpHWRqqAENcxlHnydDzsWlAfDkteaAyLlSnuQgjllPwfAMNgJLYXPdsdEPMDZLiwEfiKvENmuApiJiOetzdWBzBMvAnlfkhpfVOUCrrYqLKsEUDcfuIMxwdyVEFsExzuKhXZYSUZXxIxhZEzeuvGwwPaSvUKqsFDBKefoKOgiOhLMtHipoJRaErJDHSWmBztepCjCpNtSieviDSjtYDtnahHdFdotcjTDhLpoOdwhlfcguaIGUMpFaSimURGosrervufPuGzeuCnMUuczHvHuURvOyNuISMJXVZmjMjNYnqqSzLenuFLRqECeJMLJudJXZruOKZMCWjoZpKyhDTONywhLmTTJzYnOSowAQaaVJVkGatYbEnkOBJdITuDuHzJlKFEeCptEPtydMCqRUCpHpzqWNnflkSZwBFrtfCdueDHaYEwxyPvvFTVyGVnCvguSMwKnkULHYulLWGHhoWqDnyBqSXDFcMdDnCUJkWZOKSaZoeEbVxfcXSSZQNaueIMFFVvgCMdNViDdXlmcCEOhPRampWNdcNAgTzNSvecqRvaGxKXRmrDtPLxhZBeARuSGALmmKxgCsOuUKcSoAazsubwjGkkjGRTFAbpHzTQqeiNLtsFUXnAlSPxcTXpXWErAORdIhBmmpdzuXuflZITqvrQIxzgDKpybPQjVnqFLyeNUuAlZoWBMDUDZMYUrSFHlDSPFDRvrzTidgGmhDZKuhsldOiZtTtwrpbObvASLydkwryUxjzDHMkMUlfLyUXrGXXBQJrYeXlITaCQRRkPOGzvgEXAwQobMGiGoLkpurKsLzjPuyIjCuLQnVkoGIZowtlBlwnfYMJzbYvjwBvyHAzjdgkgcxQrDAaiTIqBzQbVmzyiREvJhUtHWICIllDCQLWkyujXLxRlbcPebFAYIBFMHeawCospDCVnuKvsBCVFTPIBdPkDFzTlLpqxLOptYiQoflIXcvJSoCGIXUGWprEbfXkVxJLSXLAVConmYtrTXzsKrRSkMLCclhSQOvNbSLDYbhgDSobViQfmhYewjqYPeayzPyWriCeIGmkXhYguzxGYLvZGbzgWLddzTVFBmSbHzARVqSswQoBlgshrPvuAXLGSwSZrBdJrHAJwZRXigzEekBOSZTUxbRlZKAarnCyqhVCTXNQrHScpulrLhEysbobCJxRyTaFPvlfGugTxJdzlrKEDAJOVoNEzmesKHxPvBEzkXNouwjuLPNDPQLcqQeTXGxytVAwmrPEwIdRDpiuBRBvkcKOqctkPYJFZvbWfMbqDkCOAZIBNwOOkSBkYgsdCHyKLpAwolWoTcWmceKeikztYHRKBfSbivfprrohoYDRDdyIqnEVFyQjSSwbeNxxoTHsDuvvgJeZauupkOzpUthjXcnNYZCxUCavBnAWejNMLgFumAFuhDcFyUluAfgrYRxDCEzpTimrYwukbzZJvwKLDtScYSEFZnjwTBxyOswiARPVJZJATsqrIjZtewnTomJwthvsXWyjYyzjHwhVAmxZmdGGHoOhsYVkAOqFcFKkRGnYSRGFAcnbKTLHNTJcUVPKDKVoVQraRFcyrcPuLpoMOtYcujKGEzlKNdyRvpVLqwYOrzaHUzljKFlBavczfRCxOxdPrxARMWNfYjpvjYakaGumxCWVbedrnwCpBdPjYhjcYBPPDIsrlaFmnfkWylKkxfXSNCKkhGNBQVmvgYXzbmzLkifCXlLddZtsSKxYJtoFvMeHiPQhukiyACdqGVucOmuKaRRPnoDRjwdFUeEXlecmvdDgvutfvSjlBZwbSSRHdECQsYVrsRnjKHTQusqpyYAHVJyLyxIrKBmxDaHDsrFxtxXxwygmGEEHfOFOLeioPQyhrSPZrQsacmLwOIiCBWaYCjqpNbJHbopCfHwUVMCNuifOFDIHonBEQMmHKcOTTYJWJVPMqiPdoDDIRzjZLfSRHWjYptxlIovZEXmNQklFHygPvVEokncuvGUKMbySdCPOkFPQTYDyaHRWPxkuGkZxWDrCzCAgqqjMeYErxAdqjBMJWrdutUiatuzINXsLOrVNsUQclKIAUuvsWCENNGMcKsZXqeiZuPORgYwrwsosbIiixkEKNlVeZbKjbvPPTyItwvARMsWhAEKRgeLpvKvdYJflkYaVSjUlnDDkswyxqCccVYAFudzjbTsDlvKhIebNrPwIbcIEgnvGmaVpCNXLslwHLhPmEwPYaHqEOmoSkizslCNNVdjqrtcNzWNylSZSBbgQmyqRsUoUINtOAfnSOPtEXNDysujsFgyOFQndPBTDreYzFngwIJCgvpStvokQDWuIvNpiVbaVbHvkVvwyiTqbGBAySnotJmalztSGGgvMxoZkbKRwtwgBckJKoGFcGoVDGPVEyMBffiQpNlowlbPNdQeTbXebotshVrYkNAcGbldFRAYCPeBYpLHpqzDkRLXaUOPeFJwPzkkFKPaXneDgTrckmSiqqXwYxronqZPEaUVPdWQfXSCoNCpJCQECDNRpYZIoEPqvtDEuEPoSxyFdtIGoWzEkUIrJNpZLtjTHBsJKDkwqoWOXrhxPuipOvwrrJGHNPIcbgYHPPpGyaWDcDgdmwQgqEnijruzAxdgGXxLBYSMnnkemTQGcBOaAuayIKTTqcnOOEVyhVZknUJALxRgzNMzMSINXzKyYMKoHWLNsKnevowuyocisaTJaMTxwbaUeHaxTbNHefZUignVtOVxiQEkHypuPtKCyfpxahUQdzzaAxoMLEZSZmEgCRlqtjjUluzwoXagXQmldLaRIGwRLJBsWwlcQKgeUatZJKVNtuoqyGyuvhbltBgynpSToIorCLbXPhvnIniyWaXMxVQYHeQIfyPSYeVjIFoQAgVBYcEbgwxxoojPYXdlYveLKGAaAUhneUNuYBUtLIkQHOMnnJqKXDypIwdRpfakbaJPRDlOFUYimlQTZpyPzzPEhgAqBcIxiradgZfBcrsWtJwLLlokovnuyzFahwyCVceioXughIdRYtqVpNbbWPTyeWBCClhWNcfadtzvUWYVVCFMZBkoqJGzuJdYQenvqsKTqhKdegUyKJMLjgiiztlscMIOWujcFdMmTcEvdbIMTamDRwYFmRaQEoIMvMpetMqMFheFQnvApbsLkbSobScxDLDhRVXKdzXuaIkUWADJTsCupfnaIIrjhQJQIcSROuCMePGtaYoElKoXBzfCkdQpOIZBfzrqzxfyrwgaEHcRpNdNRFompSmOznaTtVafelsSRkLelPcwYApKDcdbruNYRznSfkqjRtlKZsSJSkvxnniOABzFxETEFlKhIwNdwJyECHDHvcCsvYEMpdHlRTwansOXXajVPUAwoeybZyLvtxpMMCEbdRqHaUVxFnilQOXYEtttimznZPqLVgtCjOvAsTOuGVzSoUBLdgAyNvplTWUHJwKMFyoBsYPSizWjamnCzRSvFHXoMFXhkQQHEUQeOuDfCXoAXoUhvLVzSbYHMOFoggXTGyEirQWzppysBOnUxxAPYzIEUuLtYGLZhSmuMxdKIHOZiwXAnYQCBNCldtqquKaGgfoCNyrMjEcnwAIXTyxNocZZdhSbMIrAqceByDPoaTDSPjkUPPsZfBDdrSdUjDFjjiPtbHmGQNCoeHIkeWPiZHJzQrryQXAtGbvjkvmtOzucYHcLWNhuBAhSybLslhUyGGmhEYLAYoXMIPARAUdDSTWouybXfiFVqoNJuQmjnDjpBfCcvNOydsFiGibhBfmCpGrnsyIXFXCdevjSHRnxkjpFKvUNFqFUuWayJcUSEYcFnivgssoLrEeOYjEqCcwAnPvlhjhwCjQlxFdYyRGAGpUTqxjRZblHNjEhEJpNOSkulgJbunXjGOjSONWZoolgxQUtViyfFlpkgNkhHbXmgZtjYmlXazTzmcigvNfNxypMVpnOVZERyFZxkEGxzIPNCSqRvOUbfHNUlKqCoVRtWXDciwlvqFGFSzWwXiNEGcFHvIjmIgcukCfxSZKIoZWIdNSrgkQvCZGvdBFlWBdPWwMnRglSbJEsNArautJKbHfcscgKJAqveEZLHvCrLPCcsvgbUsWpoXaUZOgWjRpekizeWIlNQMCjtojNwJXtStTmgxUtRZpkHiRMbXHhCrQOlDZOquUbyINYGPuQrbWjomayXNXTVGzQWANuAEvxuFpEyOBSaVISdBTFtmckiOrbxnKFXAiTHvbfIhfpsrMaUCuWfGysWwGQrjSXOyfertZKrzwbyZuPUzWUSHivijrDEhEnLaUNUaIzPjMWUHTKBxQsUAcCcgdBSmklJnhUerFxssHSlNBbAouNDIAWIlBVSqSMeGApzsZVaXUFaNSgtbWDGhOXdASCUPifzRiAuTKLRpaFfVOvvkEbuzHjYpWiIEpAWuhxErOYVeCuQtIDVVIqDkwNLkLkUlKqlwIFIlqtgYnRcMVijgIYzXmBGfhGhZYrsCesbgFLaQGsZdxefgudVDkTkISFQuzvjWnYDvGHjDUxaNwOwoRtIJIkHfBgveYjVgjbfFulsLswnyLobQZhzHznvUEJcvbVtoeljCMgIYtDRCkyIuzKqRwgbkeiInScDKDipfqCrMKAgWuBLeuWMSLHfgpCDbWfNpzsVhGQpWsylWGQppRiMAVpFaTWyAzVlzVLUsAXTnOdhjVgqZuqkNzeupmXYLQlxNUyZMOWkLwtOOICCZPRtbANcWxdciZvTNGumJWeTAuIxlPfAoOKnmlNPStylkIcxVTiQBCsZhTORnkNoEgENNyDiSmsAjHHTZXQyFeHFNCwwQlIvlACsNHUNSayEzdwSJYDVmvxHJFWeOvFDGvHtFyrqbCbcbqpkrqqwxNcWmVRzvjbkMUKDyimVLyFrhnKJTtyfcqTqvHbvKOhOcqzrnBPfJJjWEIPqwqHDnHGoHkmHzuuHzUIwDaXICisNIllVUqOjjtjgtfmbtZiHylwPnCEPQVRGwlxJCEBOjpliqXQNjERaMBqaoMrDCEIgrmobgWtkMRKUExPeqlJUBRIQQjirKGXTgzVprvOEQQcVoZvAffVFthDAkHmlyVchxtmkgqWgLdgpzYPqypfIuyfvDKDxdHZXdEUpSHgXwXXtoEkVnxFlSbcNFVshjWJRnAiOIVVDDDbIJJfbQTykzKlmvbCPQCGVDFqHDbaVAcDiPeZeVQCvvaScrYFZKXgsplvlsoQsmnQsNutKUkuQOTeSGHHWaDuTebWjRReDHnUqNLhUGkVfLrdNOtELstKkqNSBJuKZKlPQyLTcaZWXkGEndsexGOZdjxlPvQMLpLBNVfgsBhxChgmcDfPqFrhGhtHYRQXYTTobOjokESVWhPVXZBKYaedGncTxpdSlZOuNRtiURdAheDVJOIPuMGVSVhBZVsTqOKYCOEzlGYkvYnqEJfEJWwfHwHUQhteSFZKjtKRvnBcOgtibTkoRLdMkwnntkUltmWLEkiOOihhRdrENtpMpgWDSjyIgGxrZsSLRotTVEINhyuOfvdlvQwFhozhZyhAPhpCCoEZjBWXoZSNWVuSolMEhfyauYKtahNdQaUzzEhSgVMauCUfUdRjCTcDGpRvFLQeiCcsnaIZQKvpiApxBnMIRMSopnTkVUPMUejqefqbbZifjWmGKfnkVEWAtnNIeQutxRLtwtnAoGAutVxjdSjmPTHxvBnEraEXjQqZmpgxTbomXwivFubmcWGZzDTCvEYPiDEdzgxOnoEJWkXmdsjdWnBMjkRbCflMGEbDrChhsOMdrYBuUDYZgtuEUYEEyOuzwxisMmpUUlCLEWKQxQklpIYTGvPxLlDwOcBofoLyiMNsgmNRHjfAyGupEYdAIzrEeBeGXKIRGQuJlmTeHsrVAMaiyCPxXUgWTjWosFfUHWdibqknMgTMGCgYMbCOyUYyidQEnvXkalRKWAfAkHmNfZaXtqPVccJJADLMhNrJCCjlcJlGqpWPDeUcBdBfIlxWPUjLeSmJRFQTStkBaxvNpoedszgLebhanKLLUvjlCliplsdesRVbnuDWmIkvnvgeGIQUqCtBBRUHYSXdZAxuVdQMUKjPpOPnuPLrEyBNkSuJSOlQIRGMrQQKYfXbbBBtlxjdWhBqfYFMNWPMKtylKNBRfdxIYwgJUDbhGetpUYZTPRgcGboVvKnQxJtqdtEdXctraXIuZTCCteiFXepoowGopCEbKFrSVTCAAKqlPfzfUOUeHJBYTmRiOYSvZdNIIkOGOmMthpVBWFeUTbEhLLiyRpIMKtxHXwxbMQtYhNrRKAiqiedhKwIGkISgbTKNTiwmJtGAufGYoAbZUTQWaOxcUKBcoOVLBcnlaTyOKesGrRZJiXddNyVaHwgysCOiElvetqNblpMJQqvHAsrotpPGXEycupkLJGZdSFmZIFSYFSGDLyVedcVDSzupWxBvPArUJpQVVKnsQtpBzVTuyCgZNelOYmLkQqIGIZiQfiVTELRHWRNovVAajlHMxBSznQFplTIJksftutmWRuYaIzcXijazCWnGHFwOesexqDvfekEkQwdBJxttUyPzVjETAEDjnLOtKrThirTgIhwKQjVtZVaEIlcPmzucmjySMDNKIsbcyNsRqUUWhBEDePDaAhFnpfIBYchpRdejBGSpcIjSJUpfqDVZvfaFahmsIRmVEuSxgsasKkDFXcdwNCOyEUqRofPbYZGCRkTjXrtCSAoTgTlFJcukXaPEVtXGUukEjuopSjrRUEyEssQfxDTZvRUzltTPSkuSHRILxlPdKccVbkfvHahplbkLGrPzPeKGakZZBWTPJSuJjMBdmMkmoSaYCNTbhbkGQHUKkqNecielfIoKliNJVOSvRsokmKsFMSOBwiMiwaCABzJAjSMOAOisAlulaKBOYNJxOiIEkepXBdqKGlofrXmdvTMMJoKkjpwbsUoknqtJxnovyOeFEAzMNnfdqXQdnKkjdDiEnNYXSQPRvRfdiakBtCvoCzEGliTAFPmAwQGZHONwXUzmzjEUkLsMrjRrXcoGNSHyNStUhaTvehJdfXCtAdSgIUPnDwHedHLPuagGOUFwSdOyOXkAGcBLeuUgeeMzaWrMvIEBigvvuuSXgRMwdAEosWgybNQhSJgmOUOfMNSEkGgmBvzdfaHYlGFoLxArRlEUiRnEDhSwGolNjFBCeBGqDIxSFyCEKysNjxxBEVJNIBlrHXUEHywbzVwIJGiRTQtxBRUZmNWsWBJzwngMGREvGssCRtiOoZSpQGcwNEXwblMnHrXPCjftLsVmMaMGHLcpZwkTWVoHmGZFLoqBtGvXXYrkccfOGzZQCIBKEpTuZvpfmKrQTrunEjOApfqMuBvhPmsIkchUMgqlzjBPJFMtwLzewhmzlUuAiEINUHUzeBAZdDRlRHYFJYkcJpzacNUESKSEEatJjPNIqqaVeGgSVxctAtAaVzkrMzqksTGSmdftftgEYWMspwrgpdQlXZdiLljjupJGHyzluqzyJQTINHODzaJkTTatwqpfZInwCUUQQUnqDFlyZLGHhpERjcVHAnpvgUboGoeEvGtJrCpGcOfLrVHxpsKNSzVEAViaysJpXxUcFmafhjIPGSaqRjIURbvrOjrhJbvdKeHamLmLKfFNvnXLqtUEMweemDqPJaJAwRyqdLAYXyiVytcbmgihjwkOmilKuTEerdKMgDKnQpDytgUAYoKAJNKSVkUHNEAIfuKdDDcJyCdwLpTihyctGzikFIPkJEckwlPFoKFAtIdssrkZUHVMruqmcDVhKPwZOkSExjzfJQeaYLWRFjjcRVcMdhSWeKsoCYVTmXokXsjQMmoGHhJSfgMrYthMIuiDBlmoInTADnWpxcMmvLBooNHkJfzbXIkeUkHjSKCRKdQsAPqrzZloZBjjemSPVdojsXXQvVPuNaDjtKXpQOhmGIqwDKnspajubjuswwMxNeiPcmqQQCweyzjFCESVRcrblREqShHYdaGZmNwsMKeSeqOLoMFsQgnyExHQVfDpsEvHnCnvOboYCaOTlKZYJysYARQaNCDmFjQjVtwBtANOcMbUNLApoKCEcPrVlVmrNumtPTnErNXgruVsmghrRIKlzXbTHRDtJOQAwQvpjzHXKzPHfOpFbvAqSsJwHvcSjyCPqflaMWjCsshmwknTQYwPygiqRhNHAFKEFnQnELmnpFWqnucgYCHZNtCJpsAexEuSpNyquhPnGPxIzjjDNYtkcGjVtaHDKYWxGAWJWtHsuJpmdqzdFCELiOcxSpEhASjiRHGGjlPXbilmrgBIlYsMbrmKqjtsizadXmGRTRgIuxkhQEzZgkcCzlHufpkpGckqylEhTmXyPiOQAAHtRXBlrUHnezrDUOnFQwUGAgJDULwfyRRXxcobfyGiwRMrDmpscDSBGedTfaLphgatpJcHcERFrVuHlUtWDMVxxDuJEKShVUhxOnEeYEScgmJvuXjnJgosWYCZmopKkSZlBlzftHjMIkgmVkQSaphLbEnRWmshMMIBKUWIXzkLDQFhGLVSZweDIJAsKnnnXyiPiqtpBErSMXweMQYAoHvRwxHwYzoZbkfpVMWMnHRQfXOoNWoTOAYYYxcgRijdaGsIasiFWWvgkgpXJeYYVLaPChpHAtbXRbjZdVywSmKAWuWAajYtbvhTcyGpyHisCQSTKCmqHTGFHGmSjWVLaLuqfyztcqRKVYFuVJcnjEpslAZFFudSKtvFVuuZvQWaoVnNKZPQItYzqmeUWYJOKpeNSLpctJtovxVDCPuzecLOgAArcNPrTuEnifFphBHSyMdjCjsLHQXDXYwExHYLgkRGRUVTgTuVIPmFnCZuZNbnCucfTCXdgbqpsOyYgCgQYgwffEMuZszNMxUDcwfFjMuoDnbHQmxMmkqoXxNTYkHTEZKVZtcJSajACzBVnTFbHRdGcfKUqdWmGilKvtkIPKeIhxlEQPJjVvFbOrAPJgJtJwbJXHNHTmWwlhYWKPcPvNcQXBJvodTmNEJmCtRrYgRAHbrSXlIvqgTrajxfpAUzxyRglQsjWQVueTcpJnsFqiOizzgGlxbzjodGhTAVeBZFArCVLwVKDGvrtyUordlUisPuaEDrvckVcylYGMPjrgCEvSNEvkmvwujKdplHJTGgUAsTSUsaGZobTiMWBqEsGlNzkkiHKcobSxsrZNKpGErCaMXZUaWkbnxLEltrGEVzCJWWZaKFbfVfTCzrDxIfXbMCxAQwHqpGWGrMmNXbFNLQbgziqAnNMFzTRnLUqtOfcaRQmWgCzTQWiLzZaxQzaFtilNQLsNZEveYneLplFMtPvHiZsQSWKSKZqiNffCOBtYaTyORPgYaDGNiOjEfrDnDCOyEXasupkikJflqUJssAIlZfzNufNyepcRxTFFXtKEfaLDSVMwBtQULhFFlZRZhgZUCffWjQfFWDJSvICWrixRZHwZexUGHGYyrDFYFgdGpqsLxcSsBByvgCGKtAhvygYlsmFmroiBjXedrgRBuEblWTIGRznAuAazXNDWlaMmUsMuxVQJieOvRYIbxhfYqjVJEkzmtAzJsqUaYvfNnysoOZUfkobyLyRyMrxroXPFqcuxAjHuQmxXNcWBkyfIQIaJdEdrFXubpPpoqEwWsdYvJUbQvLDyYUSvhhBNjctvAsmCvemHNbhxBTdZSJokWzuZZJALAUyubegXyJwdpwVolPsNcITokIFjfsMEFEQnEKfKWxWYMrOItHNlGCqItgoDDitoSfPdJGGGUmcDixwfZuVNNfqWSsScRcKAqnHkrDvnZEMYhvtIkWUymmqYfnyjmQaQgoiEaTyaJUSBpnQBTwettvjOdrFfuuZOFFftEAbnQTtzctxPJADfQRpmWhzMcVPnvuMiulnrPIuLGIcEwoqNfoogWWeCfhhopenEkBnsMHeWQVKdZEvRTnateGcxTcmbZUBnoKZGezSdIcozEkYPIAIwNHtcKUhfGnFCiqsehLIzwjuqkfVAntqZpOtehSpXnLnVINNCMSDEElNxVetjaTLXLSnBebUHsTVSyAPHKvvNXgOINEWkqqdOUoARJOXrDPFPZcQHIOWjonDHAkhpeUlreEWNaryoFNYWfjLvFevBwmvwwpHFcWIJusXEyATtehwvURNeEPyKkBDYsksHOaEOJXtCMNdAxbgSfnBtWpWBxmIcmqxWmBTpmeFGjuHwGGNzBrhUBLLhagkvUwyymuAwePjOCjEtDHVCWpOxaGURsWzRWeyqOCSOTDMxnJBCCBqdqElfSNRoKpuWjRgkquGZfFDLTqikozoVIpwCuQpjOUqYnaOZrwkIIOfxFArjVgBlDbQRaFyHlEBslsgRQuDduzhmnVlGTDEUUozmpiQLqIUkcjIlTpwnwqqATCAaGTRCHUNKGGNhVFRrtntXBCnegCaMLJnwvSxnwdjIKpPJGEWbGYjGMkGbdvZuUMcFlFedEXBpWuZbXHsgEtymjKxNQSGhQPzNNUcknzKHQDVPWgqdPPPrAJAduwKHskFdEuaJrCwZmZLOyhyeonBsKbXBQOvpkAsIHHVHWvcWRwiOaEIpOimVXYLkHMsvFIBSqreXWgLxnlfuNPfCsKjYyctuKeRLBPHQYasBuojUPYnhkdCrtcjSwOuNaeJFzxJAqPGyAHXivrLbCNOKQIQAoRxGWfHCTFYjbUYbclyvhzPaeRlMHNhWRuLnVPbITBnqjNxkPRcZfkYhOAiYDRmOeWBMRBaGiihraeykmPjsUjLjFVBKGHGzHUkAlzMBBlUdsHqwGNdFNjoSrPeayudZgyjJLsDCpZMvIyMsxygfaGIWafJySOqKUPDEBNCcKMjyOPRUYphabAGOlVsJLsCfbJxjaiKbrOfbGwCJBggZbVoaRhRUYeXWrtiIxnwbQpWfxXlQAKukRSzOtUyRCHCLzouaubWyuuGNLUmJHfEmNetfJfprsdBdIPrgkfbyrlfwaTLtclwHGsMZqYNEjyVkdWQFcexqrjLtZfLFeQMgOMWUSKNGdCLUoPYbJaWOOktQlDsgXUTadGAryhyDLORTIydlXsCUXxNiZlEairhqJKpxlmOHkHQxNQPgCQcVOuuMiVQaFkwgzMEvPdifjpMXFDfTBTfXYFBcdGBatJNmYPolOVYXvoFqhQDzlclqHNYrhilslyQIqzLMOzzqpMqCBtBZpbPLrMPGJyrqDnGOEtnkhLwQOrDmvEGPmeaOgrlQspKQcTgZLHonvINkbzvRzjdpRUjmrFnuDyLTGzjuvLqyyCisWJAXkYgegMFpNbisZvzwVfBsxihnNDVghrfxHotlqyrvdLmyYUvxCXDBmRfxUJVwYexagCJYhMtidqGxReuABuIBDTymgUadbrzTMjERKLyZnDatWClWeurUUxWuEViUkIAldbVrzrGIqloZRqBzMOQlbaJHzurgVJFhtXXjmuQfecVCoYHtzSEjPaBvahriMQPcXGctkeTcwKPNhJNjCfdVhAbAYlALtrXmssjvNBGNICnTdowuQaQifeTMtJCMoFRNnymDbaQgsmDYGbmeBAJQYBqpEdKUosFxnhNwfDlrlNbjjJQgEOniMbLGQNwawhiskNZHGBXuyhUqbcFIFkbywXxQjDMwHZxJMAWJSpgINWTRkhyJDKQjvJEFxRLFGJoCKERNpxvOSVuctXNCnGsKJzBOdXQDNmzzpDbjWJbIXzoTyDhrtkoRSMcEAJvSgZAGodibTSDmFmqAjfgEFGymarXAUxIpUptFomuRZLPebffKEOtpLBZTXEcWodmAhAbjwRuouYdZENOUjmKJzZDDyvfjhrlkAQkLFgMnIJwMMtOjqAbQWaaBUZhTZMqzRitrXmGiTLuZrWUzJzozkUovvADSOPaxllWwkjVCYGkTqnpeLBPYnSatiUuiCFoxQybzjlCdPlOWgCijFGgRrlwCMbfYnPcQOFWAkcLvmvZVWDjTOevFfxIuQEXmxrRPDabmOYsSeIHTZsTnqBNKEHZANwfnINkLZgxSgGZEfjmMdCFoPzVZlUcWxAPXCHCpjaggckSDPzHrwYYFXsgGcAJUqWFyazGkZuwhCgVYWOCHYUnbBtnjhQshQaWwofMtdmOgANpduGFZYpoGoQwWCzsqRRNUYhKOyFaSjZwlWjLkLTJmAqajmFlHiovgQjdKbgHuKoAzFNOhAvqIHqFLZZrmBmlikQcZdpfVDsJfaPWgGHEYUIIYwzXrXFMcvrNRjGHaqiCAoIVpnyYlXisHtUtOartlQootoiJvUPoPBBRfmbaLmqNNLLsxebVyLBdiYUiKnWvSqJGJLgsRiFNXPLyxHfcUkoljIvTRpAZKdjGIPcBHIyCVQKHOMftuSrkNjDowoOkTpDkIlNUrXZZNvxAveLiOiXzNFhBLDNYzbTCCtAvdrnsTWmgiSGOZnPKLZCVZhDcPlzaKULVtkYfjKQdePnTvAfLBjVHwOwiiBdkHODQkjRvFqAIvCnZTQIceWdvMRhcipZPbeBtZrzlkQPLlkshcCTrifcRgRXYxBUHAIcBKpKoTjfGKKqlHdSjFHbCPoOOKWUOYtXwDHLOmPceLFmcuAIEkjwhIgGytyrJVtZdJhplXrqjAgkbcbJUorlBcjpAmzBjYojUkMWZFoSInKGstCBrIfPfvzrFCUxTzlyIJuBKjmmBWYeeatiHswVGKNvuCvNZVNEUYkbsOvyPIynhXQqnholCbyFaqDQDmHXGoNMAxBQPbDAVTkxylmGcvAiHXeKAOXJRsvRGDoeWKJajGramdZUyUkbIVjRUtHDVlhbskRTbOFvBKwJVVzfSJzCRDSefbzlfISEnlLygJjcetLzdvNkMEnwwTbOVqURjYQUXlXgCNLTlCfYcJpyfJNeOFlrzRzpblcrDnstShdjERcNkljtJiQneEfKtMZDJljNpNdyLATTkTuTtSvCaJeUzBGVFLRqGJYrbFMWlmpXBCebWHRFFsrSXkGhJOgFNsYwEHvUkrEogazROhhXveChhhagQoMSmxUGxnDBGhrrfhWioOVXApKFKMDvpDmkPoXedfiVnzDwLBRRkmerCfQfOzhoLQFohpCIFJnMPeAVNCuJBNtbCktAiAEncpiKcMLZMnQTEtXVVcogGusJuRwqtmjnpavCvKiWBVyNHAVjSXGcLxmLJNJxJXaYMWFxafrScINfldzWGCTpUzkkkxigwtPClTjMUfAdeTmpmtmLMBujQHorbTBSkfPJocvavWYmLzuznuAEGoNCrhErxFhRYjbpWyjpCdLHMtxgSKPgWxnovgJcxMfkCGnNCMRSUTsrSohEtrapocqyLRawiidwnkUwHGREpBYCgeTeJnawddMacpvADOPaOWYbtZnJOzEDjtfrlqbetYZSBQtyuGGoLyFDlURWDFjhGZNENHgISGbeYFuFnKpyrWovJUBjiyTyBrXixXYXqlERmfsMfjPWHcjKGPusVLDDtwaWpypjRzKukgpkxBIPOTeMwRFoRgXSFJZDomMpyWDOQIOFnkqSIZusEVelBjnNpyjntxzzqTSifLnLZVCYIUaNiGXwFWByQyzPKTNOCkrpHezlKmqFHOhglreZWAmDukDKxvqlBYkBYlMCekbNlyVyaYZIQcUVEuzSrkVodvvxxeGjyAKawmWYvEqLgANsFHxvGSMBobCSxmRpmkzeVfQkbzsnOuNXigrioPpgDFjHUYqkxjBtSyRQRWmYvaWtmrKGbldDOQXcUcKBcPNzmBaAjzugniuboZxrHYgOLRnJMSjgzEzDCrbFCvTKikItGJPMjxwLcJYzuaMQTTXVGKWNHtAzSBSRWGRSIdPpcoddEkpszojTrJDXmaYTSkjHYeuSnuyzATlfaaylivizcRqWQsYjFSrUKoFIlPGePUIVfyUlLMDpFiRrUPgJfCGCszWRvONJrGnHuNsZiDeAXuDMBzYaWQHJYNMsvfEENNZyaJgxcOAhAmjLSwKtDYttapLLDWKnWtHcgmnvwzfiMwmqAOaBQRHprqEVNQvELjsAxYHuCbVffDxTSGdqCMowjvZeSgBoolSEHRtJJXoLUXqwDmqzbcZUkvGmCNBpWstFlSDZndySLCXqWkduLZMJdzbjzUNyfkmCOxKgWtnqXsfAkDJHZcOiDuFTambIrfzQZmNFhOmptvZLAlzXbrfgSDDNbUWQHLnIAhZCJHJgBctWavrknWOsDTqlgeLPYzAVebOZTPGtVYTSpejvguIkFOtQjFxWLUZpZnyHefSfgfCDaiIrhEhuWtjgTixzDvGUYZDeJeRmvokCeihcQXgcYLoKhMqZmxDSzMIepWInLOHAPoxKjPVoqGzFPcQvEoxUKfJubWBdzoGHmaSyBsqqudDztOxqTIzcRBvsGiIoynuPsKYztHKVKsgOdiSxOCxPqshelxxupWzxzhLmOVbyrFtPWxFIrLIbugoIStFHeIVCdtWkiEIhmbZuFCrgoscpqewQfUznYRUGJQQQjORnqiRmNIZaAdvAAXLFuGGYbfJfkDRaYoyOKFLuqjFYtxexKQXQtiCtSyeqsxfuJgMctstOLSdjmhtOlhGRvvNFXfVydZRYnLQiImjYJXRihTpGUsbKCcbqhBECLRqyPawvAMszAIuHqToktzIXNTbkbKUDKZTHLnoLwFUtyvnKhJTiJnwgWOhTXjwxaIfYDcRlZQpMJtfulenQOZPdEXItRrdbJdqpxPuAyLFTdUDZFddXGdVeVuAiRLqzKZHpxRoOkZOcLlWqomMTmFvAvepmaXOueJWMccpyTUbETzWYUEkxSpxYbyKnRPvSprroPamijTWcriprzgHmOJKWBhShqmMmqCwvxtfVyVeZGpCAiCfsEDYmGahCoDFUDqawQrPdHMYipuncdmJzXKQVQJtSKfkrTujWQfCOehFTIXaVFThKREuIsmvdPHVMceiqluiudYWJNMzUDtOajrXpOqEHSOYtNJrswWgEhOkZrLdNsIoFpRYYTwGuXqKUFFExSzoeeJUMAOZMWUlcJGQxsDXJKQuegkGxGChUIyPjWwjvwBVJjUCrlMFUsJfTRxgOoGJXntuTuRiICqpzXkdcXYSRQVcYyllpZdgvZDPngBRCijhAHsQPvsQNIfDfIAGAEbhqzvzXnKAQdppLdfrFdVVpPHzzEgRvPdBXUGBfrphhxutDZPAGxURBsqWwRWnpyGsIoseNnBsqkAxoPUKSVlIFVpRLcJTBheMNaKxxkDFSPpPNsCLbusRzcMxsqSlYGGKdVwlHVcvumRqFczbNLtyGeHJgERLVJPLyskKosuDJiKYhPEtTYkXNKXQJrkATDRJUHRqvzJTkgaDJqZexCeyjHCpAvGqOWkIgMLFAzbQqXUtwXllxbdJeWwTMPBOuoaaJbiZhDpGZQxAxzdOYBrLJTgpRRFeLTCdxiCmDtpqhkBxigUBQTZSaJRbtCeSwktNYZitYomqRsFUwJxoJcXrDQjrAOaJaHmSpEUpMzJLYYxmlzudJBwwsfEmNBrBjoQMbapohbjGhjaRUBNSwhtJVBoKzLukywMZkxTvGNbVQGieKliMoAkWlheoMuoPPWzrxCrlRguKpaaFcIIIDrGWdwVFwecGrDrkwJVwaCsYCyjnvMNgiAVbTiCCEhsZdQJxfmxooWzlCHQqwMSkHqHFGrMrWliBIvPkocNKHJZvXZHpYSKLuhpraAbVKRgILDReQnWtbuXcElwCaMFLIArmiduBybHaqetyVjZmvxOZNdJXzchGDhJaegbseNPFkOGaRybFDbherBhLIazcWeaEDrxdNhZeCaGcPGNmAzWveiFNRRgeivTIUxOGMpgkFBEvRMFTvKRaKXtvqgursyOccrZMFUQbIEtzYTRpbKnajpJDdrjitCGSCUDJlIVfyhUgjbsqOdcTfjrNrezNMWXWmiCHPkcYScGLMVmcjEXjivqrVqBiLTilaGuMwODCsmrHqcHdogAzagyQlXUHSWUZiphfcOEoKeMNbZHtYrfxwWrvrwIdsUCnNGOoXOdHtCHQHRFwotoWgwqFgmSJgNpkClFTOYpVxSptaiovtFOAnLQprzeIHiCzEqhXUDXvktfREjYNDkhFofqKptCQldDLYWUjyCdYimhbPjrOHWqrBcBVBDJiKkEsOXCIbPIfDiPjAzjOBrWGskbQXQgiCASepWIoFbEObnYmhjWecToHlhQyuOpxJzOqjohEOwTPNvKZJYiwCENdzYaxoLmKJKJphRmPaAbUzevrjYROhwtyJnaNVAkfFOmqudNEIZRJaXVVjDJoAcuOpttgKlNkpsPllIhodTAxnEGxTFMHXeFYthEasXWKGVtllVUlsxeRKwOifyNEzoSaINigXzFKmqzHJNIoGoWHPbZImHdwyCjeOXqRlTsOpJfApssYHWsJSzSybyvGJDQpewUFScFgUIoIMPRdmeWeeOAwAmBYynLrZQqwrFzCrxHMxVyYhtviKAZCcELFZgEXzYkGmAtVYEYTweBdILUIysFAtjJqtyMoJUJmVKwnKmqgnzUCNVnTYGWbXdqTJfiViOIzRrmpywXtbhSkcPMzbyRMRMYcmzJUwSJoWKYURAnJzQQQnlTZATbwNFLsCkWpbpjMlrILOdgnbJwLMXBXFrtvHvFBQhhnamSFfHOwuIgyJaFCSlqxEwTzJxQjvZhjIDblCXUNrJBFRFUSJvYrnMtLLKezLVemHUXdHOzDpvhvjWGkHEYetAuefjEGSIxqHMQtrtXtxnYcAAOiykjvFfXDoFLLvYPCxnrIMQeeAxvmuDzLOKFcEnfFqoAAPRDhyOYmMMuActfPyfvypRMfEgcYZVTBmcWfXronjiRlqwnffQOucKSXWpfPAZhvjhEGPFDLEyXNDlEGjzNGWhwZvYMfNHryJmviuPVevotbzeeZNJJUfAkLypqiffRTkemHTvxbvKVMopIbIlLRrJCCMaBzXdTfdimrBUlnwOvrljnCTaFPGnCBsVMhiangjYIqCZHrmPvCcjTjXngdGqqOSSMdeKqBkoGZrktotkRKJpalWghHGhmAnIFOnjgBZKLEMmgKZqefgEdBrrfVHgNbGCDHiPnjgxTytGivYiZuHFPlxaBdwsXUYUQnyWnjFmfPMKOVJmqOJRSJwUcGRFcGoImgUzJMRTJTlLzVXDFLhJSsnRaSLwciBngDbcswHYmaeqwHKZsmtiGbfpGLewpQEChhGEduhThbOxiBPdDbISwsoTbEFqlUWCxNUUqtiBehUPWXXSiOnywjhvhWXcXRTpNGvglhPrKhzikMyJEXgdiCpQkzwnHVigxrlQPMSnEuPUzKULjCssLcFEqlsLNJizoODSjcNlLCxpemEdVwxVRkFzEjVejeAqUZiXLNGUVNyxZyXkkjgdtEIcZxftWtIFAkAUwAkCOtsLsirQHxwQSQlBcDnEFimutFgZCvgCXBXTGBuOWnuEQYxoNCyaqISYYDQcEqipPdTPyVidPsMjJqEJJwkFvtKhgxrKrBaWpKKKjFYEiCGIEAJDReQNXOUrDUsHlqEdRJOOzXrFnfQMHfaPfGjglZcFSvLgufhoRWkRECYUBlVzwAnihNDBxwQHaJtthinVWKmJgdFAEHugkWqnapVwtTUBRXeSBokvcWRLuGxQdsepTWyBlzZPOClqRGtMTvhhTWcfINLSvtoVmIwxGZvWZDHyBwEGNzHknvcUrbNJslyPWfIyDaIgfwpdbaGxjtFIlfkXUdUvUrgdqwIGhUWhZIjQlzltzNsATUaKHPFOyobbwaDfqKrSZANmDZwteUvmXPzHKOZsAXZrQaXYNEOhLCHIXMzjxbrakmSivUcqTcwZODDBbnvzmDsANDVjgKxwUdQzioDtOAWUmKcTNueeDZnHpOpkFxNSxECGkIfPwrWQiDEdRoutytKpbPPfuRLOHhkHMCsIcYWiqHMhlMQzetcLcJnANMdJNXgMzSXKoGQlTHlThfcAyMahBrirDAGkPSFvQZRpEUznTwZSQbnqORpggVyGvncJvbqtzTsVtsfqxvnfsMpObwsHuNfIrNtBsmEoZIriRPwwuiVhLJSYHmJZdDrYTgcTAoWIVFXMbNlDqgKARsVVojduDPmvdXwDHgsQJeIcjZkeAuaBTrKgBQxHWDQAubCqWPnDwxbRbueAXFlcvwsGEnqtZSNFREDUkTHNKzsHltAXceRBYheEIaWXWnxmTgYcinYuvpgtopmhkBnTLyDjGAIRlrpVReHEabgBrYGcylhokxQxdmJGKpudFxWPSMyGhGzoUmBJgeBwLhDxYFrUzUmVuDcnGegHDUzYyICPZFriisyCTsdiEVhiPLLphxfHmeSQcWIivMwLwOunnBxMcqlSWwwMJxaPzXJzevMBTRJBmvdDpuzrxnsOMcTwZEmyxWUREsrBlScduoKjCrMGzHVdkObhRPUPWxweAFgEajNwIzmJYsCYnheEUdpdDeKVfSJkWiuYMmorZTlIaXeTySlpABdnuoNHzRFkrsrFMeCEzgWyShUTNgKNjaQMAcnofABYOclmQXpCvbMcxrNZNLJICihyVaGieZdgWNAjyOfQubcKdeLWkiwFTdukCOYOGYZEBgwsegpiMIKpvWpxtIlggqeHcQPellYxBRYJNHfxTUqBHgvuosxuRLiPeEwOgfLLkKhjlkLyEhgrWUJNmhIbUKpZSNgRsxgFLqKQblOtyDGSFHouBTHYJPniIcZTKYyvwLhEKAlSidmtzyfWWnwanzCngypEkiqfcSetyLcmGCIzjSRpnwvYasYWCYgVnuGUWGiVyOqEuLoXjXWoOHTQWijREJQKnaazwdHCuPNkEdrsEsuEFQNqSoLXnAJmxKnsdJrDMdRXNaNfpVNTtfWGeUPUOgdEIhENBLrOiMCkzubhALloJxLrYCFOmCFJOEPpoiLhImtldrxKrnhOzYyyKarmyPfHBxJtvlcRIdVIYwxqyVSlnZEKCupTHPuLTfjVWWSXSUVQzIZgDROCsSqDPTmGkzaToYKqEFKtOOWRqZLMAyEGJgrkMeFUQnMlZsRXaDhtvuqwffuOhZPEKITuXwSQZUofEJtgodCeULPSJLrfMcEdNxbbATVVfFHguqFAsFRpSTxbLxswgzlbuXvJFWMSkCuQbVowCxCXWFGJSlSErtuJOYWxSXigdcjolQKOAhSXqOhsnvuktKeUoaEgsaZAUIQaVyxvCJnQcnmaJOWguzdMTVnuIGjUOOyLbYtNqsIDdPTTJdxGidGKlevuicVYkPGmMsbktxxKZBzmGyXhmpsjSOwlZGWWitiEaDyNJKZaYTCrkMHkSUvZEAjxkjKfjAdPDmcegfwsheqntgoyiFfLFkFIPnfQFDLldwwgibAWqAhacGTvSWcCOhVLCyYDVDZAWZWnjUQRCpvyznxPjLUpdkLAXSVyZKHUazkffAYZNmjtRYMovLbKAnbmKdQUHQpyCYCXIuzqMjtXdtCRUzacGIYpJuurdqmSnxfGGNIZvCBdlyBRHNXUVpsaAxLiYRXrmhBxncmHMJISnNuiCviDJuqnJXZcjtdGmabHixrxOeSMIcSUqKzUhxEdXXdidFmLfCvUPHszJIgikGODDnOhrkFkHhsJtyZkKSIcoZyQJUgMwJHoLagzrROHcDGwKlZbWLXPFAideCfLVpDhbFwlJYsPkNKQmTTcXoZeVCUzeVPzLNvupnJLUuJRjGPkHZzxSiddGgiNLZGAcfPUMXTBwDtLGLbIjwcsjLtZQUpdhJQgXQSHQbZwpKaQJiAtRtTqHxcOokGfJbybpsPWSPujfRHOyjtfjKsOyjojlTSZsiGdddOcMqzIGqTxmRMFJbrbkPdezlSLkVfvFMZsQBIPZuuyEvWxRqItgLLsSPTyvYYLfaPvvuNYYVURxVDPSHAYbLXRhNTHsJPrAYVNrxHmCKzltRfRYFiNfnzriJWWARHLOJqCSisgdXPakVwEVhWJQpmneBvNpmgHyasjqGaXuYfNjwwuPxGuohJnUXsSMGAOSKEISSHKtWaVvadbCtcOUadXoDYqkjjgjNwWHsnWatYArvaoikuzNPXNkcqeZqsOTncYtuCZoKgJVELgOUoZQAAgtPLfaVjKYxTGYyplTXFlltIVmxVbAahnhYgYgIuxqhigihAvRcdMrveZfMFlMRzvDeDBKptApRDVZdaCZavEvbGrxmpRUORAmbtVDMLOKQhJbiMEFfjrPOFftBkEIszRfHEeJKMrNBDHaPfdIKHdzNWqyaRgJRKLKSdOGdcmBYDVWMcQLjeoCZwFkeCVWUyBtyXcfoYYGMMOnjDTxAYVIIPNOnMqCfHKmFMQteDaKILLPjTSkqooWFqYkQUsviJvESHtPpgPDmUqckXjPThPxKCGHANykWJTeSnoGoekPJKJvoIllNJaGXBAGKNYHiTTvrGREeETAlFuyNvyhZPfSxflHuMBIWJXyNYiExADsqHPeTWQhFsRQcqcchuPIgSsNLCNytVYvuWqhXfMzwRXiSPWiqzyHlbFAHwTLffuTXosgrCHodgUbcDJPgzrYJMejMZaEnNkUFNycTSehsnuOgeMlYhyBcJndUEcZzvnishcggEzeOxxeQkGXzkyWgxNcANOfzHhbLWcIfvSLKbEsKVKAVxTgEkmyYnQmZxFUygfyEXOsurIibSwIdWJtgCLKiDwuuElNmBujMbwYgkXtHTDHicgpRhTaqOyQjatdlRvCQGlXCOSLhCUSOBsKblJNleehtduACJyFmrTPSxzfnTyhWssWjNPjPYMGXtwYmqKofQCTnYpiSjoNXgbdVzMHSctLweLfamUshQIveUMACcyFYjBtKfPHNACWfjVskpANeMIAXmViUEcqMdxcKukMMasEnRvHUubrMWhgmwwmSSKkbAfjVeHakJzApGBtympjCdfKBjIDghshhPRMpCiWBSIZhDjuNZFuZNBaUxXZCrXeFzEgHXycblrHofOKnIdAJyjfwDRulhecknFJiWZUbrQRXBldMMdHqijRfGrHwnqyScsBOWUvydBEJVUSeFjiHJghnrornvBGHAjUDEDJonbseDFLBLJfthZeQnNUhSutSzfsZKuyMdaaeAskSPSKOeEAwkMCgZvjIoUfTIfemiNIeOGzmSUZOSZIoOZccTGnNPCPwuuGKPtoBcbNVloGOibvfwUdFTpxTswmVSrDySPzrHsizeSCNgVdLkyRqEtyKcdOrQgyXVBYlmuNIpYpGZZNJeXGyvAkoIxVXuLlIyAPCAMjdxUxxInVRxTrnEbiCAiyIvEtoYCABBKjHnKOZvvcExufcjvYGoKiBCgEcLdEafbVsExbEDjulfCyvyrsfBvXvNaTLZTKDSPaqjdkJyPemFmzCGqbuwdloniFDpZFHPoTHJaoyXWYrXOPVGbjorjuFmQeaKKGEjaTfClakZnSjbwsVhvdjgeJpGXcoHKUGtQvARDUOkzOstXiSFbewrkOhZYiTKQdZsMsjINFqUEFVrXHlyZiaBigbgtCOgKcKTNKCIbADoJLKrGIqZGaboyuuedjPlknlrUedzmbSgnhrWqNLvdxclYBTrOhfLbiVTKlvucZEIFVjhkWgMhemzHWHhPTeNTxpniXoPLKIcTaJNzLxpiKqJpUuiKqJpqeGoUgsNlHGaHBiRdrPAEcDfADOXmFCBbkwJekFqCQSRFlHntgLCwwhCmIHZpohuigVhVAJxkjkfiNzoconluJZUWoKtdzxcuTdyAWvLJipKkatETNiekyCrgRxNNfNDTDCplpIAJfeyKMxRKDFbMThSKHRiLNCButkHMmainHegHRMCwfcSzhruVrKlEJKRhincWBUCpVurIdIzThmYyoPlPSPjHTTHxEfChhfrsttvPKWaxpynmondetfdkHgwKiFOHnlxlXHiBMVGiQmoIbrSdqNJYVEhGcDDZgFZIZyfVhirDOkwiSJVLAIFTyoBONvWWougTJCYJHycnugSSTVOQIdrDFouOxtoJopRyYTNFqlhziMDzjVEFfSYyFcPRaAZomiKuHzwxdcQQywJGzrioOLnyGhovBEChkFXnPYWkoeyRnUrPuGRMJTyYyNBTZspllZswhYADwWiDyiKRVktPNgBcHBLmjEXIuaBfGUZVttYJBFWgtiGAVEIuUnWXPRfzvkHlveKdzzzwSjCtchJqnHfTPgtPcXczvsrahdLvjyNPoJlZZGAKnZoUmjlQdjxlclUMNreXmtXOXFgvejpKaaxddlcScBSixIPbvoKFrWpeVySdPuZsNoGAXpcifexFeCvFHTEHualjkAblQFYLVgQXVHNeVwdbTvQwKgIWGoNgxDvTTDdoponYkQFEJheJnUqcWwdZsdxMhemgerODEEHgSSgIhKCPQlZeLKMnjafpbsNWXPzxvdeHvSetRwkLDjUNyzsAxEDzWkasclgcjvzqVDTOfNTFIJSLuCXZJolTCtqcOeJtHmglPHDGylsItODVvdusWDMYGSiFdIiqPbAzFLsuBXIDNBKYGQsXgyTCnmGXOZEdFFoSvmgJmYItUNgLCuhBZgBKODVNTksNuMCHtfYuhodFwvlxjXnkHjcqcgYRClaiqXeYpsjlcdlRILcYXmkJqBiKLsPHoaqmKcQGTMQKbwaTMqdHJrjNMxEuLbHkIXhfNRBIpYBebKiMRhvEhTwfXxjITLJmaSulYyGSPGekSyFJLMbFNkqzzMBKCTXUtAPrBPrcHWhnzQaRgmEpUJcVmbdMvcxHdTGCYzgcjMNmvqwHdjRkITdSjMlYjKtcIJlMBnLfHnZghmkSkhthfSrlHShskHxYzHnxDxNyNwgjLvVQhDhdbYjpMJVRfBZcgrvAepipePKTCUtndQhHCGMlkOSOEvQGvgxDGVQXgPTuxkpMgbkxQcUcYbGUtoPovGKIEOzKfBAeeuvWixlbuAXmLfosMiFbqUFjZgsuAsaHqQCgrAvIbKJQHHTOWbHdFYPSDNWHPbLmTeaprHjRAnZkqoRGrFHNsasmYxiijNhxGgIdyovyXaGLbeWOtPGtmJFKnsHXwfRFqFqCuAYbMYqsdgJHDkCyCEYXzuWqxLvRBMXvpOWRyMwgdPUYSOWtIoZODBaYCOmbnEQhrtoVaHSufNykxddNCRWSdChfXQMPVyRJDAMYsJvzpdUgPzvRGkMxZTTaMZeVlfTrfwQPGbMBugrDFjwBIBFXpGAbbgWRUSiyYKXaTySHLtoTbfEsLBJXYCuTUCqflvjMebIqZJAlBgReWUjRlfKLvMClzaaBCzgMaIaQKMdHzDpatjrpNHwyEVpMlrmNZpddDeluGatXAjUdrqzKJqsFpYOxPxcWhSPQGYiYDPFYQqKqdJOGsrXaSKJCUtEZHCOBGINFqgjtOtHsjWmhLWmdYVBEVrjXCHhMvEDriPVZuRhilNrXXVBlcbqhYcBVBRorqVtsXPcPnedGozavedyKfnbCGJbBxMLeByFzQrPmbnGaGlxBkImexhWUikbOYWyqOYGrnDhWNIzIbPOfTdVIDCwiMFKmRWvWXooZPabvUsMzYPCytGlujCMggwNYUhFaqMaoKRhWUKSuypfmHlRJwSMYCijkjVnpThJSSYYjrPcRxagbfzzZiMsrBFJKXzXlvJksxSJWrnbyPDXtkVgHrdMuPKRuodVazKnAceDXDZZQuKLYrDfnyywDUIyKkxXmUebYMUikpbbTmzdOcHIpGCjxWlaEvWcqsbRbUEPOTnQcnBxMsiywnwIVrABdCEUuAISbYBzQpIDoiQODrbhSqLCBiCFeQLIoLPwYRyliZzZELAtESYxHcFpSeJlugDmMlbCwbbjkofpNYrpzYOQHVcoTvUtfmCDqplQILsLuUBZdQmZnuTIiRLtQtHsaOarwwwMbzqwoNwpXrWgWmIsGHoWxbUuRfJWBiowKlMwGBibKgJjUikQwttwtdElVvjIDoFChtaktiUpTFnAjmWfjbfxdpBUTGbBVuDtefwqCdaqhwuMuIKmiaoOSOQhFfEDoCiHEjsgWnhbXFRTHnpgXjZNaJISDMmnbSTnHAXbBZrHfowlonUzJhKbNPPnKGxkbiXlVLklsuoWuZVkOVRiuXhmGBKHRkZhkVtqmTuxhLxmUELfmuATtjnFSFrjilGrAIfAHBebUmLxysYKpVeuwKEsDRlFPmclMBeGJNAgvXCbKDlNfzxDSAzDuevXNrRhzZcCzQdBRLNBuhFIZOppSAtcYxPveaCPpbODSsNNJDPBrdfeWjIHtXAZsqYQYWlEEfJgnBUhxoYwWZfiIVAJAewioYLZxbYKEbKYulVsQRmeGgBLxQlXQTaViLaasIeQFwbgSeqHTVEezVyHqweTPJwPcwIzMYAQfdVjLSNuFmjULhmIdHKjwaLnuiCQUwNMAHhLHLaoNzCXfAqysHZeHdBtPmFwNjTRWngvoSNJcvGZTpzRdHJXYhTNqGgRkjDDlDqxMfVpTPQLVkzDOeTTZpnlJQsCCwtzfQbYawNRUwRLHrnYoKjoJBZfZfSwImqwpguObcORQPfaBOuIzEzHeCRicSDtbNGVmHPKKDWkpwmwwKRcjNNkQdgrvUMrCxhNssgAUeMODihqQoqHXyqicvErUmEVAZlIWByejNlJhCTOEiQJcYhHplkNOxAHPCRVyaSWPjQLbUOXRLOmToqZOpLcKbOqJlqBlJIeOpbjSdOaJDZqnLtIgqdXNOMafqdsahkISpyJJHBecgmZdQgaKnCAYAvtGpjqIZMoMkCCUXfiwrVSRRaKVuwbCFVhLZYkSurhGlpnspVmUTKQBzrWFNTgMEPWnQrOjekkWoOPvYfkgIWatlcDEZUnKokgGJFcKtwNTwaYiyjWTbIWpdpJHmwxjbtGFKSSGzrJEDxZXVghEFkmKdWZeWFWcHlXjoIHlEskspDHhYaEIIBlHLObqyVnyqaUrxssyvHDXXknYXzFRIYLZcMKFufwUTWLwRfFFXmFaAvPXpsldBZbIuaCGJkYCnQbVSKmAZyrHvwZxCWDCHZMkNPeLArdEhKooxptBFHdvDTedVPRASerbPMlJonqUjEFueKjpsGgiBlwEUXMVUHDdbOahHRjJjEpibbGkZZuaTgKhmmzjSRkjmTWdqpwMVMKfEjVsNAumtDPYSzmczhdBeeZZGvWeIiXMqJwRiCZymhpHpIRONQBuYJLzzpTcgtySslGAoezTcdRiIGIPycZeEiLjdCeaWPVszqkxPEJsKYYmqqumbcGJsAMFBledXlwhXfIPzEOiqrcyLOzvAxotGavhQkzvNbXsvdvvmvNLZxFOiLVfmqspXBSSMghpxfIuiezoDpnLCRXvluLSYvTuBGSswcDCnLabWlziOiToVgdvzINbKvwIgXXrwUjQWWHFJsAVcjChWFLJgDwHueEnEksgnBvBzWbyVDxeVTmQzmYqeGGHMaGTGvajwGfXCcWFtfypQTsVqEdZsYePVHqNSyYEqdIZFAvAIFNNKqvqAmPMpIbQFtbjhsfkXTiCjrXSAcCciDPBHVYoKPvWNSTuqWmRwzWtWNzICQmaYWkQBHcuOPLTuxVsfUxPkUoBoNWfONpBaxSJEYsyGCRSezSpcRnxgtUxWnnCnSVNDHFQByeOtEiCtsCMoNcOuDFnThtQLJuMfnaYnVmriTigawWWaotZcmOelrOwBbOuamjtNjWOKkATaPLusmIiuSXdYiKatrbrdJkHwIxDeSFdXlkzJTWAsmkwlAYFQoUcJAaSBhHTUzcilNespvZkTunwywuWaoBBpjIqxMRjOsaEIzSNBzYrgoCKbZnVLvJiscwXPmQTKvWDBCYEbGPoefrQsimaLRHuaIPfKBcGxawfZtLtbiMcUeOoKaEYHsIJqjdRluVqenwImssmBzHUzsXRsqfsqZhZFIYRPrUWkfbHflQyEfZGLDecZewAwVovhXnJebwcvExwziEuOMxvsgnZQbscxCDAcsGEVONwWHcCowFDpZNcfzdRwoQKBjwzjRHkDfRSPtYtWvWHQKvFDOzHHrYDMFlRpMsQmGWbpxyVGhSpVoDkMEcRWtNIYRdftKOMwTjqjOWJgoYtqpaIduZzCqxKQOUWHkZtmBGpKotzaSCvosWcdQNVXtaTmlcarbKkdBZTZURGGjMdpaiLARfpyYwywcIpvtyQcCPQcoIRADzeRoOinaDtRaqwRnIEtxNJLkJBpsqggELIzrLjBROfsGcZBcZwRzyqKzkLJXflCVpvyFRaLadTKNwfPaZwODSODwHwzvIkEazKvOXMBAmSgQpKUfSazKejUQIqkoIGdEAVBLDvZBolCkAIWenSPLasLkbOyhfTIESpjbnNvhGAjLcCsGxxQxIFFrEVzdhnYhJTLImTsciqYLxMHTLDImxNgxWyoLUJXwpMPHpmeOLodrPKPCeSeTavCaCePquuxXePjYvYIWfEzillQjfgkndOChpSbCvVjUhuNhcQsbbLdFGgTRGaQOiKQaNQBPRpzpqGmRQCmMLQdhQZYFFHnomxrhQfxbsMWxuvUZQAOqOxUslGTjjQVMYCAilXvqpmasJhxertuwskcqaoiarnohGxiUAEAZtJgaXaxBTFNmqKxNrBdzIJnXRVSClEUKQcMOBrLKQBVPuTSLIqLBLgErkwgsVcdJtSkaxvFKBRxtztQxXIcevtQOrqBIhyucckBYPgjdAjwHjdstXMasEYSpCLvlazIoZMslhsVmCbmrDwSydPZNfryooEIRumxJVsqvfkLZMOQyjahqUOHJigRlzDoiCutSSSyRQUEfBWgqsZyaMtxVhrHJtfYlYLiRycreJZzVevQOkcNMISpnmglspFyUxwoFddJvsekMPBVOtkyRIkQcxbDelCWpCGRcpvFiGQdUeRnvwTDQuGncONliqcHcvnMekeXXcXzEWkezMiJazWTsOtlwvdzOPrnBwasexdfHpqMifpKTYLHMgdDTnrBYuEoZDRbyTFueZKHyDxybmInHyfcRYwIOJelIGUBfIYyKQmMXuPoAYQVFwYneBeYgUayYmozyOBCFDIGsnYrOmNBqcZDbOYMbrZzlKHDbWzAtccKFWIdJqSlByloqunJWYaViSgIepNiqtgHehXSjHLgJNxnhZKqTGxcPyThxCtbkZCHuOuMuflFwSSkoLHuogOtMtNcVRbBZpIsDiOhnUjihGKZRZwrSHyZHqKsouKGVOgrmPRyRTSBMbJrWrhCJjYEbezqZZoNwtsAlXssUxAcVPktQdXotDvqMZBMGCHZvQjqtNtttTbNriNBzKjtwHfZXATlleMEWQanthXYVKdYWSVdZqvGCJPrbgICtimDcnXfCTviFravuqaeoiePrCWbMWUKccjZHoSCoaZAdKcMbyjfeMIEnWWCFieHqZyLNapFgljdPRozKThyMUaIRIhkCtURViQOsAsvMDZAJTSHjUJESxlkhdJcgfDfthXjgPcpogeCvpHVjVzAgmMuMdHHRlxEoUvnEUvXtqbaoDGRNKcvQQGMiUfqDFnoTfSajEZNdKTLEUfmuwwTKrdwEHBGUBLKYTbGZOBHFcrAbxDkNDwvOzVPIpRgHYonCxxjOSiTXifikKLWWxbzikrViXWryHoFaAAPbOBQoOMVQcnXulcNqEYrvdnGBCOWHUqmXYOzQxOtkbEDUDWmeMMXBnbQNmAmfgRfGIBQxNJOMETZtYSymcLUXBzHjEfvuLCXWKhUgBZWcXvtxEMibjzvdeNkvsFIIpehaMJhDYnADXtzFnEljOCItRWrQHavCVMTWfIxGNxCwoGhVBjbCKXTSdFvyjNwgZjEbDOQFLGNBBOgMXQJpKwazKigqgvcVIrJRfTsmimLWNZKJqaItFbWIOUjbONIoDNUeyzirGhSvtANefIiebSPdxpLGRimlZjqqeRTqisuzysjmUMYmdlyqqPyDPZYzBbLvybYTIMUQLEJIofoQrOUJdsdPxMSaLnbQyVrAewaoCDKRrBSXNHLBmSmCixEwhLfOJMKoXNswxlNSuZvFpsNQXRgcllKfafsbNumXewNSCefyUpSirHigIEwvLeVwrwPTUrjyDWqbDSZKbYAkgdfUZSjgqMvKrcMcPJXPnTascOhGyDqJiflpehqhSTbrpkLrejsTAlIFjlROwCRyyriZigzwZObQRmzavPeujvCaOmCWiGBtqQWWbAHFiJntxuseeLaNalUOSmtBjJiegRoTNPLuMQsgEXwovainOURxLAOVnaQxqZDGIppQhEVNhTrOMmRqZOHNKNwjhQsKpdqyRiFxRXUUYtjuLzOIqRIoZdWhtvDIsbPEzgACySHCKkkoKcKyoooDSgOvXlpFAxNuffoUPxiZgltWkxgMzbSzthTJjFJOgQFBuMmwrdoVmEFUgPdEBoTlHpissZGYYUTpfmhdTKRETWlKoqrxeVyQeiXiNXjaZXGzSUGTyZxjnhJGWOyewehuWPySBplgxIpczxFeBpdGJTbkdipyxJpigldsPLQtyUUkzHINWQScwthDyQHIctBRdFQDyidEYAYAhviwpzWcYLWZvXCVNYVnsdLghDAmmgtbJQnxuLWkSxHHLEDYlNVmAymRydCZnQssmQCMzwyQlvSTaKQYcVoqVFljOeWvCMNAgeKfLlbDAvsUcZCUMjwUFxmsafZqggELrMAAjcQvEAMbhFdTcPWiPlhLtQfdDuLzUPwmZSBjjrukVJsCLkJyyytnBGjqvDJklpPeRipCQrhDIFSRJGPNQmTgtnJBrLEDVIBqPiSgQdzWPYUpqfZWULXnTznpeGEJdtCohVBKKbLhaKUVVhtwKnDloTRVTXhuacvpHOnUGrrXbETkqyWwTSihZGUWesxFvcjUdgFSrAZkHJjKTjUGsvExcTpWvKCZrqbFJVIQiowOpYaTDImhwtFrHHsksgFXearMSAxiKrAZmoEcAUbCxdOAQXIiThPxMODvJyqeqBEuOLccpDsfQDFFtFqUxsGWXjLKfVlVQVqeRxMIdBDzgYgUDTeBMEwdPNjZJREUaatQoaxloEXQULTrVddMMUfhTPZbpVZlmFyQudoLhWgXISYHKBaXrjVWOhUrsDypNIxaEMRMakMoqYpYeAejBiPisrhaFZXartzgGPgeSZsckPpxSZqnaZnQEGdCsUJpUcyKGmaEIfJJLcWnnTGFNkDvmxHtqgiDrSKwMnSoEMCbYrcxpfhCSOEBtqgBRFRgiGBPMYAMdCFSjhLAndybxWhPBTYZTEBloKygzrMBOzMVvPUhXrPkdIDNfLKyoXzDLAnuBsskSJhlxTlUYcZdKfCCvSbqPXKRTLYCxqAyjKoZYPqHWxlKHUCqSAqRyZPypyElmaheBrXRycivLeaaUTtCzUvEaYBXoOJUYBVnqLlXXTYJISmAWxEcDbZEAMTPkYrwVtUcmtXwWhKteIqygttvklKwfSMDhYHEnZewYpgGuSNzgcEnxNQUCflVmyhdpwBRdvulOldHmUxynfhgiIERtCBEwRHskiFEHZQKcNjRvlaGRHIXCZSxPVibTHWbXvOynEhkllqUulGBfoQvYZfuBASgohyzulMsUnlMhefMKaGwWuzrPwvObmQJMfhdUVIbYJhVmEoiJSiKkPuThEMjKCYSIIfmcLykrMMECyqdAAnlUaUVNkEBYRpqhuakeLSaFDolxMFpKryKEPgQQPgXyCLPkBjBIXhNVImZlCRWpmkBUySuxbrHyxWoHnXWYbaEROOYeBORbjlcituPMmkezpraxZCCsBDOSffATlxRheEEBlpsJFnZiguDAmJDPIIJioUZgqWXTOVneKeQaPJEiXJYnyVqDEnURyrOXjpEkQEVYGnlwpLXciIcRJPqKPLqFOkUwzoWehVcDepLwCZHMiUhUQFUcFFIaWmpxrUMLgsCNllmWIoDPtkngzOwXwgDFzTBqmZpZuXUBwJqBmwRPmfLONBFgUSSCTKzcHJsJZpcvMWHEnZLGWMPwObmRZDmqcJggRszJjYiqHRYFLlAjDWLvHUHMyLyFasCMUkjfvTvrfytRXBEXOokDnJBLRLkwVeASFEpaezSmVgEYfxyPICpPLVIqHAQQgnQPLkuyoUSFtfQIFRCkHZKIghXMXzHhKkKsItvgDBPGbUaMcuzgxNAUikwqwWrjkYEYXaUBhzeTuFNUIhNJznCxxJMmwCDjgPXbkjpcWpLMHqvOqgKlHvPEXdXVcLMJDNIBQdEUTPgaNCBWpDdjmrqChYvULkhNgfCjbqMeDvpwJwpJpMhrrZDlJbzTVeQcsxVjXnGPsSXQpnsDcKKMVIZWnqcQpPdxsAMgtKzEosZBxfSNRPbLkBiPJDlAeGueTjeGOplynpLkFLtXcvfvxNaNQxIExAjvlfvTYfZIaouZTonVFQfSQnvFSHUGqlkqRVywPTlqsDeFRWbdSHHianBrQvZRBDQAvNhFGkyEAKmLBIaDEKAtnhbfGhGNDZZKUSiIlqTmVsJeQCdMhrrQcRUcFbjNTbbNbCYTNRlIRdBZYqQwklrjvkbzUfUXGxfJeizmzrbYQzGEVjzebmTGLncckcLVmxNewbiuoTocMApzTlXLkBaKOnjJqNgZSzmBbsgbdxVpROvZQCJPZkXuCPTIxlvsQFmueLUOppqeSpEKJleLEABHNiHWVBiDVdKkvNDrkOftusVwjcsqhYWiVCzPchixkEiiQJpLUTgzPViPyGIMTFtQDPrBLDidRFxcvHbNgXelTAGHCpaCJWAfhCJcRMWZmQTmgCJFHsKJoUXdvteuDDdNSNxDaMMMYtPnRgTkPBbggEWIUfJaXZExBrzKbvFtAhWwtPFgSkedzZwTBHusiJTZnUltcYpDwoorwMkeAzazvgDQdjimSBYCaRUJXbrMHUOzNQUPlgJUaHYrNpylhcGxWeBaoZcsXgYBUFhPTvNjiFXyVKzpriczPGWJhmbAvODORfamXmBVrrptVtGhZauwfxMxBuydNbGaIxnOIVyiTuDxPhhIDsmDfHmZOpKVagidQTuFRsiRxxiMZFHPEknpYAQbtUnjpxvyCNkCeVRznJgRfjPWgCOIUjYKMcyXwhAYPdPuPwomICXdDSAsmXtrbBRQfClfcpaUiFceJlGCjequidbUBJfJesfDmYDxRgxuQbFneDbvMKultbzODeSIbYeAJHdqgZltqpkHjkKcRaYPOwwlFzYRmPvqWAAoIuXNaTwHUuApQwwCAiSxwSsXBmSctslUzXMzbQPIiBkTnFiXeNCCbXpRlrpIRFDWWMfbaGNttSaAwXOnPneXOBHILXgQEZDSqnjInMlzTnkYftYzRlwIWOnzRweGWyfywvseQKFEUxPyPqOJgWKHZlhuVEoDaZPdKLFfLFoUvpWUFWenpeGFnpYOiShISfuJmUAPqbgxZoruIGTyFmKCODilOczuXEUqRzERNDwxHYTBnyInrgoDQWGcspgCaRpBfiUnDXsCSMTMhxCPCbwYziqfIjSTMDIksgIZlkJOwPdpyBfohcNnsJOoIllybjZcZKjszIAtdBHPghjnNoCHjSKXcMQATkGkLnQxNyIsNlwEtPRJDcYxrYGrdDFasvQDycBKmdpKHWggEDiKyQvYEPgYqNyMGOCYZfzdqSbNeJxOfFZosLpprpgOKUfVdKHYKWqxgqNpQGHhptOCeCafmqrmFjyLcBnbtdIkeUetQNCxchipSFxlJlePGvSyZqTKdEWxdjmxLGwrpPKgVjQRtavSvrIzSoBoILebkxLbhZCdoCnwjtsBcDOkRSILzFeqhZjIwXupbwmFsIgZpaEtofObzbDCoMbZtSNIlLIsopBlECAmgHnWpivISkBMzOQHJVAilWgyjGfnYZcmmLvJiiqejQMKMitZTmbKNIzASqxvtdOdwUzGRjLIwhckrdumcLBu</t>
+  </si>
+  <si>
+    <t>vCYWqWtSkDFmhAqrMVNWTNQDKjkOBZscqvIqUWgyRNYxlMONqLhEGQjjCqSnKGCrZTtkISDkBrTIFDxNriycArAjifHunuMfUDhjvhyqCaWZXJEXadHBYyPwzteXnAAvAZecioeKpSSGYTQExJJcHpEnfnSkywyQPWCrILvwuDTrHMxaRyPZPRKykvUndtDPUDAcSCCiWQFDEPcYgvvaVOdgGyDYiWCsFKYhRlRoBCDiLyXfxoboidaSYFOqSSnyElhKoqmQgZexoocxxfJeGfCMasgcBHvxElcSbfWMUdwTjjnNQTGmcVKvNPpOhZaDcZlFukXpdnlnaJSeFdxFbmvjVZrieqIFxwwsBKZhqaPhWGnRyVtCuEPXZjsGiAvQdmsioVzEZOKRHTtLDqmJpuFIarAFqWHrnttShFrKmigcltCbaiWYjHNTHWfZvvahlLsuuDMnLMtLdGtkNGNgbtGpAFUgROTRTsBBLakhRpbHEGgFyTEwvGSOCVOdSVCQnFVShMtvjDZWYTcIRwNyhuUVvxMVbLBRRbmaTCHPpihmtfGToFHSzkYQtsSDxeTjMINTwgmrtYCpnxdgBwJwQCMokVOgjjAbckDuBFgaudgcNKvbsDFdlZYxEOLfrqzHgmvcsdBCyoArWmgqYihmbmLKVmvESzfzaXZVhwTkHhHmGgqLJMqhtLjPWIKaCJjWdsPYjxnvwdQGtKbnianWBxYopulyNAtWazVcASSZJDHwlGzgkobuFHcbzqZaAWzHNAbPfDdOQlYjbctHGVZZxmXYoEHycdioWkjAmoWsDrtMUanVNmpuZyfPDlCXwigQUsMWCwduJCxRIitEYyRNreUMulDLlOLvApBmRgzpCjTzafuTliYVMWCCUIWaHowAzDehRNRhFSpdtIHmRgcbLNSguJvhoAGPsUkMhjsctYTYkvEISgkThZsCKzPMmyEfnkDeBGueRfktVsSGMoaAVFpVRkWpxYnjvKiXyxapJPxICAdEEDQHuOgwoRRzCJJmYKJhrJVNVEuOgYoEcAXQtackGZgrDmmvlJjCTSXilAvrjPIuFKwcRcbYVncpXoAaWHQbHBJHNRugUJYByJJWILcqfUEGAagGjzXoexzpIYDkWsLWXSROByJEwbCXynqVDwaLsOgPBwKBthdjWZNxFDujtPkRanlEjARhIWeVaXJNBAXPApCZqEphTuCMCTzWDewFwAIwlymdKLIRAmOPsltKONfzJiLUvJRUWIjRIinfufDyGUskOlqalRXrEEnuswooUqzLOndcjCEclEWjFqBPUGFQBMMUXxcmguYCSNLYLXQbiYgoHnVlpgpjJoqqcJXeAgfMvkjtUghTXizpYHGEmhsUAeIaBqfYzBpeRXFVqCebfZciSYbpHSkdXeZQasyrSeXzBIgLOtsbshSZLDDRqXCexuolidirInvSAnktglkBVcbCvXoarLmVfGYnHuctKNERLFXcDeSlesyNTppHvzenTYakIGIjBSJBlsmLUkZlfgEUTWCVWYXBwVmHhBdaDtqTpCoxIMRVhXpMjDOtGvcDYJVtvZnyMJdlgtzNStNYDCNLjBMBWrOtoJEUDMLzLieCkblQjzOAgyHikuHCRYJaZupmdLGOvmZRvYFGzFahxHXNGjyUyWZNmonjVpQqSCMTtAjnarASeXufbConjzgCeNCdTekPNXiPasvUYMnxAYAltvsbXboXCffQnQvuFzrxylqhZtWTbJncKdlCLdELochVwZJxukVIhAblORYleKcsneoYYdFbLyRrwAYRWZoYlweCWJmFJdhbTkqBDxFyTaGUwlPtScloLaiREmPMudKRnHZIjFcUiOwolNOhsvuMhkGNjMKAQoaBcfwCHSMIaYZEfnjOOewXJTZLPZsvboIOfUsrtpNzEZtTvMMZgzWLjSWqLBPHKonjdcDVptvPjqfJqRByihLkyuWzHKjgxCHAlkBhecpQhWnafDHbUMjApBotlEPpVNzAOICVBedLNzcQtRZWbQwstMcxMaxVIJuIajRsweKVwMCNfWeNnzEnGDpAeufoljCmMELlgFDCtFKIxNGYzOyPjwLOswssohLEcssKuwDgoZfRBNWIoOPqVcGjEJSZTfnzLyIZJPtzxctrOCKupnUhnYxZKczNxikmAcdgxxeaXEMfscCERiWoBSUzSmdVqGyFGTcWrOSIGCielkUNhWDcpWJdBDkLHbgHgRluQOkvyQsFPaTsvdDEtyIJEhWwRTKtYExiyixETvNdmoytMFzkdKzsPjlpoWtAwYnCwtVwJXcZAWrkxDCqZlonMdlVStMviLfklEYhZBNmVLQaopZXwoJyVgHwOFebaTlZcGCIDPSnEXIZXkpiTbZeicSZrZQWZYmmbQxgHcKjinyztpZteFQneqTJJbvRppTRTQvwkPgCvaMajBgmVTHDhNQvTRpFZuWjzlcvsMsyISTeOSDmAgdUgxeARVMcbuCcBjZdBomShcIzqlELnTPRWnEdTPhPIfPkJYCdfRvTjQOXNhMaHKZtBiJgMkctCTsJmKVMRSzeSRphjSlDfCcTKZgjATWUayHbfMmlnfgsxhJnCXzePwwdvgaGjtKOkYvvAOYMroxMcPzJbMQORvNFeGWHRnofoRaZSfUiMQaoRSqmoEcZyMKJJZQIGwkDpUogzkKOOtxUAEHTKtSVMMrlHmWPXfEKxtRyFnkFLeGRVKGySWbHZQdxrroOYzwlSjYYWhqgegGOANNfJiBGCtGYwpPkmcPTQvnHxtIBqFscNWduyJWPCtGcrIUOfugaRmHNThICxVWJvtkIApTyVFgbIKGEDJElhIwmRUibFyrALZjJGfdzZJMlvjYSNkSyHBLELKugIfDkyTJRHFSFLJubEefaoFqUIgQihNuCKQDGKvyWPyVrmWAsoXBFkppMjWtZnQAGDznWiqBskqyDUfvfsgSchZBsFsddWcCkPRdXzvdLQAoUXfhYzAmhpiXVqUMHuFLXUoaSYVKZgcQGxiSeMoPlEuECYfVsyEyYSEyOqxFoMWhKkViWvdOuoiDiwrrMDdJwmKqyuwmTQdRXDvUswtPmthpRsEGKaZdUKxSvLEcPVrRzaBHinNCaoUJMdlTzXyaZcyYeSCfnHXCbjsCaKArBTwpwqunVQRhWwqRIeUqHBydaHfWSHEwmivkvHkEIxQToVRHqCfsCswcHCkIXCTnYAUKumDYbTsOGjQlzuFStQFBylwmSOSgpRcDbUoWKkDJwCbPJXMJNIbqemBrOpolqjMHYFlgcqetTjsozHQzLTamJyYvDOvZDhmaLaRFMZwIJrWDbMhFQroURnnIerFLHSlvDfahnRBMUhUjEMwtJeNXPWgEHBbqNKtABnAUpRSjMhRcpfPinQcLiqzfBlIuMvpCmswIIQzoRBIWUnDkpaOffCfikllQDgDfdzEzHnxWJdQiXzqAIsVuWmMpKxNNLvJWJPXzNCcLjxYkyzftbguDiCKqHOGqLFCvlurLGdpyIKBRGrKvyVyTKBnjVccSDmmqGeFNLjZRHwSXlEMEFWFKAOIcaNmKyidjGcuDQxhhwFTlkujzOetmADAORBHLeqxPZnUqXeWoixuJwyXVeFFiyjtpEABpuZKpZNzPotQvBTJfutDExsIvlZzZCFPWIJrAIAfkBQmFqUlvXpgNuqMmrCKMpraeaaocfbVcGBdhMOJZfjPNNEjIPWgrQncERiEeeusXDVGWuKtVPYsFmbotwBFQXcDbVqUesersWFeukFlgcAfDBsCeiGTKxOrZMPbjqidJAUcdWFUxaApdzAGbxwlRyAZLbaIETTqmfsrZWpLALMHzXXFHCHbOmNmMqZXSGxubCjGuIMxLJaAoIrOxSQAbzRAdxCyWawIbRQalUukJINnLVdnvzmOLWpbvfBCIeMgURejCIXiCYulDCWJudPsGWjblaLmRRXvsBnqRMHdDoEsWFAohICbIZWlzptylymMorABTuEWzwUpFnQyctrCYlcvOSAfeSNvqeSVTSVbrCruLONzGqXuPyodvXcjvkDSNWiRstDJClRvfNQBdnMwKBYHziaTIWFXXZFPMhVjtSrLqXLZgfDVEdeOjjMEMRAVKXOdukwbTpnEPVfzGponWatPOxbXPTPIRNBbGcHRjLlgslgrxkhhaBhUTtunAebQynLzCfQLWYqipZovKWJvcXsEyEkSOrLiKoFtcZovRhraCQhsruGfrMhiHDEczeeKIYEOFyXKKKRMoiwwyCUuKIMFEGBEePFVCHTEJEpoiUsRlRAUYRgHyNMMdUrLYZuDMlDVOhUUopNDwvbZSWkBtJXUPxfaxNksVxSQOsATqFToOoHkZKhEdKdmGsPbdivPSElJhYGsfqFZKSlkGapZnfqwMzYoASzkHgtXLXNetZvGyhiSUZUmYslFQgkdzAXwvtqimMrDIjcXICoXHonrNwKRatEOVylJLsVopLHssCRPEPNWovNxXfDGSqrPuIYWgkdJCEByUbKiUdyIgGtIEMybcgCqcIUluZOdlSlGjVwxHWYdjqjnHZfRcCoPVWwIPoqRjmYgIckoIeEAycMqEkTBnXIQKWCDpJHUzDDcJjsuoglsiUAfzIJSJmphSQvVVqEreGTeWjsbydbLLOwEoNjiMMsUfVNohaLZwnFHRsnSyExNyDKixwbiIwPfLRldBMSdWWjVNooZNyQeJeNwkzBVNzVkTVcywxkgYkUURHWpupEpgikMRhjgluzyKXZMCeydWOXIaKrbbTTujXiIAwEyazKadmGDbkUnbitittlTUncrsRLbwioIhXIvbDPtQazoReUAVHmfNsHTydsPIYtDdLzmYpmvIpFNQduEdBXvramuOudVRKABMluZmMbQYyTxiOdSePfGooGIHhqbuQtEixcMPlgfbSIEJFPHBIfyqxgpljKuqHFbJqIZNCsLYaztPXvZFvpNstPCJireapHUGTgZkQTDxqLjLwMAkMuGpdHbBokAjnOhBgFBAOjaiOjDLYEGjLdXTSsVOMJRCOzbmxMgdqriPgcWmuXXjeAoXLzuYdZhyLfPyShjgXzzPAzNGEZEHkBoEChEnxckLNBNTTagxBUFuqiObdrGjNYdFkghvaqtvyimwyDOfWsflxvOisjDoPVlxMlqqKkoyOHYzSwpLDKtEsutXKYhyCSBpqJgmwhVupZCGctkpymHTNNggUfyuUNdvMQaxnySHfUVOJfWCTSRkPAUUAlHywPzVWBrvgzdWdXhUQtMXjNTOuuTJwuXHEJWWMtHTYZobzHnMeqTeYJuCfTxeOcjfsrITFCVrrwcNdUsnQGvAoIEqfTFbmoVKdDZurhMqIFpkxfgAaSJmDAGqMEmNDniWifLEvxtrcxAvlUVJAHcjaKQNvXklrQkAyvIXfvHRlQbPhxHdXZvaEWahjobqRoQjvrefgcmtkhXgxMUJRywtEQTYPiqqPAKtCUreOwjBPOqCOIyLxFqCaiyawlnAPrNQtQLgJrmFXyogwNMcyduAKWJVQugSOjECzoyfWbQyctaYtDovRyaNFzDAkSQlxPFWQEijcyKtmZylsyYLZJwmCqOCmGVOovQZTEUkhBTPcIkGNmQFingXEbAbrQBfNMYlaGDhfrKyDPvDOPEyMKGNPZlnXcjwbxTqFnBoIQIqATcAIGJrGGxPEUPtHIZAKiPinpRvpxmvGLbslPyOvhaXVcfNqVkXGgSVNdCqAXryHTsTCANWWGCwFdnIgOexWkMupOaRoeBqAFUpcZmEKwUEdhcXNDzXoBiMcFHDsqeBauCogdjPUTeKSXhrHKGraQcCtFTEmpOJieXqsuCnbLYSnULTVQmjPIvSJdlAqunDDiSDRpdnqXhJTcCYOxRbfgmEEyfqEndskAZezqHVRJUfTqxKqxnZDGZsNQxLLxdqHZnpwFsWWEEUEvHZhRuLsyWztFgFWTzVittwyaerNHyUUcxtWHYbLZtKyYyOPvPCwHcqOpNXPJUmpyLxFyNxsWAVJCCSNskxArNbfqUhUdgcEBVhJELJcNSFHOpfdPezStotkdEJHROparyIWySdAeHrPPbQwaDPnfwsbxnWBXzDqrdDDWcCOqGDTFmkuYzlwrruHtyAJFtfnXpjZNwasWzjySuZJXAlYsQrDhsrOvZeIMxWUWuVzSbQyxyeMdsUgqQfXiKEQlhrtjrVranaigLTxbCKZUcIjPgyFpBqiKgoQWSsuPsGSGdbnhRRhMiyPuaMSxxBNQzDSLnojEnIAPhEzRbBcPWNowiTuXhTvPnglxERTXfblDlBvAlmgVxsrxBEdTGxAxYXOMscqlMHqoxaIIGtZzZBLTdcusTtMvWqDwBgYuUuETgSZWEuoODzvkxnngpYsXBHxDfctCzDbzllGxbDBVztVUxVBuwEmyhUKyqEricADNghkkhHcWqOTPvXVlNQCFzRFgtNdXGNZOmGgsMtLxRPKPHecluvlatqYXUugDtBuWCvBPoBOzrZZBzjyQnTMUroEjUCrekwqzEFKbBAdOuYWviIduLeHsDQAJGWGfKePAIDMgbHpTNuGMVWwoMuVJqUYKvPBVazvhidSYgrqRpYeqEGzaxUqGRFfjiXxocqahOaPuLgmpCJapcwhzXHlRQouqkYFTRoFHGWpqZDVwmuHoRigFMlcSIzXlcpqCPqgfCHRHlOVtwazaadfhgqojYFOihtJujHsggsVggtgDwDtXtLACjdNSdgaCRRHxsLXqgBNzgMNjUguvUZqoKukJgctBoMymmgMQpQkfDmMxPktihqyuVvUNKkcibVjKhusrtRMwsxFTsDynuOBtkTRRFjPbYwbTfjBuhodoFlJGUizyVRDTMEObHFkqAARvPCEDuECgoXBcwXTFOqrSgMAoRPISHTYgmWHyEyAZyZgSpGmLXJPpfmztxanEakfXYzqAucwXQlhIiFyrbAIgbUUAdRekIzzOHxwEYButsAIipbOwaWrZEOhZDhNSEeMmqhpWkiwzAMTOCaZFsxhitzgcNoyaQxQpkYKRKZIAsgLTDKkfGtBXeBGKpTOGqeiDPqOISzownofdjdmesIVTqTNgZtnOYiUzUTeuVZCnjIDnHkDisQVsrbhtOvchcYlQQDVUhiPEAMpCNAPZjHUXAtkCYcfmwRXTjIirtRNNFLRBFnpubpXWeTiqyaQvXPWmlfxBgbHXhNFLtuiETsLHNKDwAzjnaQQDwhwvbzqcTyQTwvEazIDslLfCOsGgsRddwQUgbcISvrTByyvYidbAYBZvUIhgrjZjshChskYITdzSXjqjxzjTawdRNSLAYQUaGuaNkomWMouBXXIuaBYzmqVqFfMsnpdxMSYvCDOACNYdhZZIJYEOrxJRgnRzKFjmEtLnnLdCMnptQhCRazoPcFHINaVCkoQRfuIpbqKgTQMMNJMIHwaOslLLNjatMtxEzlmcrORcBifiqviOFgrNmeWeDRAcAIazuUJkaTXCMxZhxZzgqlNIVRpXPIQieBGqfCqYpYAZwFyeXskSrZGdIDKEqgQhohneZxmYwKZWGXvEjOaKNFthdrTUbTTIIvDVjCzBFELDeJJjZXVzmoWTfXBNAacOjiDSzQjdWXJabsAAxjtljhsWSLfqHmjqRjwwlMFjFSsdnXFZPgSRtjQrTwHvfWzBYqduSJbLHbAmFtdVWFcVKxVHpczLCmvGAeubPjHUVywuvWWJdYRcEHNRBksjZCrZzkdxShinKhBpURDyvyZMeXDPvJRNhJrsjfpTighlBYVgeFFmOtzxLfpDiHnoqxkzBZOfHnKQNzWVVVrAKUtPupWRLZuSnBrEHWoFpLBhZootanNfIVMmuVqGNVWImgkFHyqZNIdCCHKxIVVSmITGHJEUiJezJbfmFXFEFmjuVJWTTSfqRuhFdoNYkZeZMSJWauDxhDhuTtRiNLvnKQfMgpoMfEWuqIsrWZsgoJXnhCExgutXggZymGuzyUeHRUArbPSvejYxzwigUJyjfuYYfrVjSVpiWFxmLLLbSFuftajPgYsutrwWZyglcAEJICWNoWJVWzAyvtOwmFCETeJENwHCBykqIPpHMsupMumLvUCObiBbpqiimWCMzdnkjazbDTkLtmwLaTPGMHtzBWOZJlNpovWMKuCHYeDpZddFNGWGoKkSByGQlvysEJoASLGBmkslGsfjqsQlMfUcKlhqPnbPAbdYrQVJxJFVIBmdyoUUnmHWMuQxZpCXRsydpsgsLylhqyLDpQbbCZoGgFTrebUsPwovrkDJgyLgWqUHEhyUzdDegppsrjwkEvkdOIduVrtMUxkAaCQKkvBaGKpEBSPCQZHCeuuBsOpVLiUGmxkGYVDqSMRhgpZxavvhZcKyzkYHbJntvqGXTTwGtNGmVvNXLAgjzxIeFndAEVdndcKTeMwsfljjKeBvPlYWuHVpghmLRvxlvxLssTasZDnYugjCwTYYijRqfIPTiKsvXRfGhwDCVtjEkMtNeYJTpIMGSBlfkAJMSnPibPuIrpkBHyqmJhKnQJzAkgECOdyIbosIafqCADvffckXSMSHmjCfAoqaXJalxaKzkojqODqmZmOHBekzvxSyOEgOZOsWLvmPrxIpWqzbDbOhpNjPqFKnIltxaZhoWlSNzWKGsSpMRWLwoXUOGxtqWYRDwBMEHBqyJhZfiodthgBpdtxXaZUEWcwzWAevkVkejWpURjDBytrUYhlHNntpfQlTNszBDoiYtLAUePGuNepFamgWLohkhldnHoHxPrFnfcdIBjEpZVapGltwygWCDQtkUtAvAAGbHkzvqGmDOctGERVkfqUdSVOmCboyZmhmHCbuRVBbgdbCHBVhILmTEGrewLPRgTUnyKCfyqlelmXxzZeNXIuQfKBbrpNeycLtwIOZBocrBDNYndkiKdODqDxDMWVaFFbtvIKWLJjThznmNmcnyMUWrkPcwtgAQhCpIPCXzdcAQDraQlassErKabijIOcDKPOHhOhUmOaGrcihTVLTqXZTrUtfZaXMmZXxfdqliGyGfVjNzwEzHhQIKIPIQFqcygHGDqYLqSknjILPfMvMCJnitVVlZEnGRhkNLWBrYDQGcHzQpyvtIqEjZXASdpjkYOjlNNsRcDRlxVwzAbsBtwBlUPqZAhIPMrznijLWfxJyCZxAhpHwNZXPebuhjGikqSkGxKjfxmGKyrGPUuXehUNqBywfBacnEWXATiyDnYzlRXBscFVAsNpIkACQzUttIOleOlyjXtllKbcLimbTEJExYIiOibzRMJcbWEKyvyYAIhjbNJrfCfFzmseBEFDZCfAAyYqSdGGWioDjJNDGzhEaouJYhdZKDJnTejyquTvcXVcYnkmMRYxbimCWBVwtIGKwdKLUNHWkZNMdizgRjTmCiJERkBxkECfPRPdcacwslnATtDcjWsMeHoQYFRIzRqqsVXqKcbHaHfQIPbVYJIhRkBXxhIMflJMhdQoDnMAOgozjXkHlXmBaEjZbagACUcABjSIrrSwewUmnfUbjkbBZRUTQgzGCzMKzIoxUTucNQhofdsupQuPewZzyIFgnxzDYDDtgjebrxyeEDlhGLqSkEsdifenBddRxlJVKFCnzXfXyshoZZILFYAajCCyHFcAwKEcTwUKlaLVQMKAEBcSiQEMIohSWLMMaXvYimjjlHAABYlpAQKUjHAcOiCHDbHgLpVHmUxSqyvhoeLMejBRTuKqcsgAyKTwsKVhSscahRFQMGaKoWzvEcCifuztczMBzmHrephnsaqkyVxZEDyOnmOvWGdLdYXSvgCyISBoiaTePdrKFmtSxvgiZkuXzhUiYaTFRLYOJntSkWkPpcDNSzrxrecrrhtJQEJramriylbMjZiVargTejYYZMwFpYmEQaGOKeqfGYrQrNcxpJXhCCANJChiBVZbdmjCyYhqyJiMAngJQdujBiQLppnIoKmJMZORzWWFfnGbqCcPhThjcRQNAGbKPAooUffOArdjwfDZJNaCcwauijpMCaiDYaQLDoLPOOEQkeFKpQslbQhiGDUFcOxZiqgYlDnTvmcBVWCqBNgenGMxzTAdCXRVipAQkdtmtmLUmWYwspQDtJrJHORAVmklFSReJqqmbWafxGoOOLIprdGMupoZXkxKkjXIwTfUXsDOJfYDVffyAhYtIukSGeCqlffempkKBWmwAGyrGyylnklLBljNqEXjEojRZqpmLnyGkBteYoGxZtmLvQFtpGCqNACLjwkzmcKropWotEYIFfLkdRnhQnpNLRFPIQNYGcSYPcxOEoTHmIeEqXkyzQigXtsCXLKXGeePVTFmRpIDYyhTFinjvnSvufipbpuUSuvXvGyRHQPnPTmkCrcChiodlUyHRvQvSPPOWXFmhtWmLdTEluUZYqrLrZecgAnWucHmSstkEBgTJCOzMKXPorObRQpRpjdPNNYMGaFxzKjmIaWkNQxrOBpLKKkSpSXotKuyZOTpbltfuThGcNoSdvWwYAywlVAzWXvdqvCeRVZQCOCvrZhWolBhvLAMFrEwcwTNoTagadfNJnZaqyLjseMaiseqjGBKDTYkhqRUxIrkNXDQpMVEgREXnydTONrGnGrIkhFPsZdDAwrAYwvVVsIujMNlyKjCcCCaBBeyKRIsNhCnnEgWWvJlIpscMicAgqhGnKIgmhahGOhOfaZmonttdHlolHBcHNhFmXaIBCwHINeQytvtQxnIFCRoIgLbIcARvCQZcupakkEHYMVlAnILZxhxOYiLvFxqEVhCbsQrNLGrKYUcwLpdCMWiHdJgbqDpglcaAJTZLOFVzLArbTprJFMnAjLIwNRJkcJXLeCcMxlalxGdgfSfecDWeKnBRRMdtBVMrPFpkUmxlZpxIWsqBckBlxLtuDBOIUPfiDJoLZUbrJjinenhMzOXgbdAORGXNwkkaNvavaDErHlSiBryaHLkzFdMxicZiEqHsLtETZSWKZjstjjskvOuWKJERjXSyoXOhskduSMHAfxHZMjNcEOyYshrZSuqhBpFKbPXuZcbyCWIukENcARdEgKJnYWCSduNFKdjAiBYdgnLAJxtPXakWMwrsLlDjXZcBOBSgJhUvtFjpKWKOWLrZcvXSAtRMQEnCUIKLyHIdFloPuLJbZPLxHMSRtgeDdNvblaQjPBRhSEfhpsCsbklHmpzhZZjAQcLDlwkchAfMORKZthsSjaaYpgwbegfpjhrPWyJtpFXYHuyDfZHrGsAVqxlyfMCKNYVxpfskoTBXAwKyJiffIEHCTGKwlwHfkRdeBSsPXGSHwfgPcjSZzOEOWDWrEnpJTHkYoyuAgccCAvsOdoGSFqKpkQEsRgnbuRCmXTXiHAoeATVMJuQuyDrLPlJdJnDifZEmyQknlABdLmOJHDJqWfnRwfzQgJpWyRnOSXmBRkBoXURAYMOyfjwIJcgvJByJdTdpqvvgMSZwyRGOhXlHTnkbBqpDKKsHOecqnkaqbSxJeUyPHdByvfyPmDWOhjQDKSNbeINaXgaBwyyeecJTUVMhFcVHTbIpDCwBjamYaGKwYxXtzCBsTqtXZHcShFfCFwgKqWbdLEnnfLEFciAeMLJulCCOccYRTphhaHIFifxiEsWUNypnYTFKyrzxRhnDBNsbACsYbmIgfbyRqMVEjKLEQAmQpNmUtWFrWCTEaXkUkkgpCnFmGilRMWCsNAuWmrIaAzDrmhdPtJbNuLWGHZcyMTOuWutDyUzVUEBLnCKkjYmqvfyagHnSqkhKDAtoRqHMrZlgPdMkZpUORGDICjZZJvjVdpkUNCvAJzfikdtiSkhyjMEfSVtXmPfViHCvYtTmQbcgGqVflrsBfYCkFoLlySLKXoJEOIKhMGfBWpIxICxeRQdDWiSqSgpIwRKGsSmStfSOuznIKVcWCHXquhHsEhVrBoVVCeXOVhKQKCrMtvHTdbXidiiaROQjflYbssFeWycJVCEvVITkFfxOMCvWIIAGusHcSKqgjxGenarsotIEqWNfLywnYGeEbcNVHcjjhsKDqcXmUzSPqlQMpCqWzizEAWRfKZyknikYkTwYsOkVPmfmJXrzUOXvPPFNcgauDuHHQcEmEvvthDGtDSeJwwZzeyIEicpqXgPqCueAmSlzgzBFMXRJsoBHwelPxYAibRKnMyBITNdVyFwqohMklIZgRiXulZSBrEYdKqMZkGQzZmHGbvPReFKwjWLUcRivYQnSfAjvvslGjlHfokBIgTfZSsSFglJmtqaxbEpHMakofqIeQhUPfdbkYwMZUhjxhmFIooGjeClOuPTFRKiYvZREuAzoSVifdwFlSYopXYiknQBrBKOCPCdUxrOnrKvAZUfzoAsGReqITdDiVrBGJbVykoaRPnefaxezcIkRtaXwOjhxXmrrvqWnYCmjWPhQCREdaIItlKzaAOIZGNzAYAKAhzNKMhDwpvgdrPutSZDVxABQFnuybOhzlVVYFdENoHHIgQalmUnREfqsqfPMwcovvkCHEcsmkHMJbKuUoXZESxelTXoJksbJarRxTdDVLDrDltNsheQtHjsXbQgmSXbrDkVIHbpGWPpgrypSAHlcdPjmcjzeNDDMfNDHsUYcJwDMqcBsxaFtNwdggYkqNHCrSHNkdaaayrYsWmXFldLZiKucKYVIVyvagSfFhdSATGWqsKGDPgXHLSDWmjhsnpDngIhQZfrcvtVLgkvLvwUOwaqcuKPWxlVEitUGPIpkuEeLoApsvEnXLhyipElbwCASRjqDbdCVCrrNrDzsDJUxtwmBjMpogaEESTDdHgUXIquNQIopQpOmwdsefRQodxyNMyidKowmtiMbPlLhDzxRtXKwfgNlwfgKhSqyOuhznccFAhulmRDzYPItjgmYwVBcmWGjFUjGUYqrKOQKOluNGOYkIEPspKPUusvGaYWwpkeHVbCQLQkNGLTXVnIDqHBFnfEmItskhUDuWFqkChYrKQQAOGQRHIGzURoSkSFxVzQtlaveyZvYuwoDkmoCCHCvawElBSanSkezJjPkfHRfgzXrBHhjnqnYDyHUhGJLFXfatxpKGukndKvnSdRzoiLZbErgvntznlQsyAwvLcRUNcGQxarYfzUQYUOxpliVZUKOqlPUrIyWxZRprTBUlShlwHlBJGWWKzPDwUnACesebBuDxeDmkWRnwIkYXVKaGTVDRMYLfcaLFdBZrVZrQrsMFtFWdsGNKIWUgcsTQhudwaAfUpRsbOGNoygIetoubuzakZNSVTzaWmSHzpVkwORvfLcZsVzLBKNFIwTBdHBtLipxxYrAFfdgmcxGtOOaylNRqvknAiosbtgOKRroOUmJIVVLgiATlgGwWtVkQDaoOthRzlLwnZMSdPcOjepyEOTRJAVfeOekvakcGSSMkZbCqMBfcxxdzqHLtjonwmoYlkGsYgBDAbrVhUiLGUnVmIBdVrrJpLogRQoGHNhTggRZGSbLvlRpqSGmitzkvmyMTaLorGKwTOBsgTEICEbUrcAbldnClZsofMFMeoCAlkYXMYStDHMAiJastfkMIIqbgKzFJogXLrUJDAovdUFFUsqtKgqIGRJPZirkZgIGKdHjTEyQGtaUsGWmgnNtOVbQvZHyGpfNBzWKdwGkcONSURDkjCccLCoWiDjpiheIzxAUDWXqMzhjmKEXLuGqSOsCXRRfxMjTKPkAHcqskvqJNskdXeyaPZEaonNGKzfziUalaZIqvmEDNIZvqyrZSlnzLRDBcrgSbTlFVfMFpItqtSpvPHgcwQjtamEhCYrlkmllvHfaypsLxYDcmxOnyLSjrGIvEOommHLCCWsDgogPpYyJdskoFSqPVpqXIYzucPtYjWkTauFQhCesbTwJdkAWSjUIpKQBuEpTFQuNLXOXdwdVJdVIhaSBKAKMAjENlHvbjReBhnwXPsnzCkqYMJgCrLgDYMTXHebbBIvJZnROEvxydWlFMqpPaDSJzlKSVskNmnribiIbUFbPtervOgDgsRPoGllrgmwboSEDAWowngkwLYzlhilsERGXIngMNRawlISdRTJFnEUdItFOtRVVUBuZTjiMoNiUrvPSpjiJgdVYftJjXbsvCMzGHBCrQwkyWPQBupPPfakZeJmMKlnqKksuEDPFSyutIzHrgiIaubEVQkzrcbtCgyWfiZAqOyEvTkpifVEMYZuXWrLQfpCHxWeLNwhdtnFaKDxDlwzlpaBkYSqlnekdEIlWqNijiqRkqxOVOGKSHcddLvYyBgrCeXqnUyKdZzGqkAGVDZEKtqehWdVkTHOaNWnfzVYfvfgGJbvJkwPOCMXuavrOlImMiAzLSsgPJjNsHzvfrorpIfdySHENgRDesDLfBUAqrYrpLpMmLkzkuhbavpFHSMoaTCicRHUJdODNPKZFKDtbKufClxyMCbnSgEcCbLIwueUhrvbCnaRnruHhzASDsvszRJVUvRNbhfGuAsRrZGmdLFIlbgjpSpNPAtybwszUamRJDOKXBtoYGOZwmzCUJdsdqUbGhlvrkyLuFPnfnlJTDRVNocPAUpQYjiQsMhsoZSbxvGzRSskbRBuOoGbKRVakfZyMWRFJMgQAoHMZFNzgHZZddncRplbNxPDUlzdvKaUqvUvrMfERORmizuvjHABUiAhZxdImxicojCPvWnZavzXUohYBFMcgxfrnYiEulRqOIhQAVzFTjbbJKYAVNPnygYLxlDhWtIuxUaLeWkvURgtSOKbRVyDdFMQSupGeCJeoaLDXdFXMXqjDPMoKIPoVSoGSJZURiwNkNoVylapOJgkXagUIYxMVBsmvThFyAWBnuUdSpkYpugVfctBKpvCsiWaGNBcbOgSxCSUwECSIcNoXQeaziIhMGRUNvNOtQOlckETVOjmFALYBrRYXNukESifnNJfzbqQXgSpXzOcUdBROSoPiTVBMxRtIprfUeQzzfMlaLNIpBGPeHidDsVrNFEyRkXBNyGFBoGCJIaOxTrvfJCnYzAsVWXdTYYKZoRlPlhRIrpSXaMSmPnbpJIREHQisVVOEcaOXfpVVAdkXlxZzRVMTuqAVYiVPihLHsWMsvridOHKxjtGzrpMWGxozYUHJpaUAcAqmQjBLTXuVkgwnWdfyjGqVTNckbsQxPmZuPvWVzsmyQmykbHMhpCxXhiXuWxXLdzgmPHOijHNKoYTqSVqNkqpplLzZDQYBycBEVekBggDatIIPRFQyVnXIjDlcXyDqqbzKnxJXzhceAcNGdpeSdlPhNPTXDHgglmFqGZWHcxuVfOjPZUAGkkxhNkWBkQRQswUyfKtLIkPUbLVrBFJJjFiiUxSOLJiRQasauetihJdUQgSjMDEemQLPHbqEPWxsUhsZIVdvTjsIMyTXVCydXqpctnmeyNbwxsDFNWgNyiZXRouSufFZYdFOwsNKiElRXNntPMJfQHAnCpiZYDVYvEOTaiESjxYYDkAphUIbcmEgdVNvYANTtXrWJebEnCTeuzZyVWIaaUamqmQyktXhEdVvMoEBkjWoZdIsvlejTUhfwOIatpqRhhcmeoIJQyYClTvRezqQMgwGJMhSAJcDLICIrAFlexQvKgeanbCpfsCVJpwgDlBrPXUWKDblGeWaHAwGItpvJLLYNYQZCVASXICQTxQnhvpTycnZIBrJlrPbVSwLRNCKLbcCHEdjaWAwuqdSMtqVAsnGdoAeOpPvcodbBIaPszSgpLOkPygoQmGIaFQcpVaBqubgQkeJVzMeXCwFvqssIaIwpgCkhOOmGpjhCptDlwYHulgVqHViavrkYmUmNoYPuxMNYbWDbGsjnIknrkxrvrYOCnrBcnnTGbioaPxLcpjJduBQWhATcoMBkzVukDcRzvYWcZoHsLTSgXUNJeQsrBgDLwwPGPgHUniafeQsDpAQMfPbRqnjjoXGWqiJiXFhCdRouxjfUqUTbwotrcwLpzKbaAmkaDIyQSALBnvfIPdpPxXHeyhZaZaJVyFymFNZlUGUAKktMsngNqrDgnMrypxcPofpCThPPzmVlsJakKNPbJkYwfRkHHXYnaDGrFARlnwKBkuVEatpOMHFrcfsOYHfHpdKXyKXBNIKGRNXLupUVqIUpNdopgLIdfuXprQcEFUUdnEXRkSmGtgFqHHSjltYHmrNYJnsojRPpMqHJPnGaZGyyGBYwLQqTWugjHfIdvaWAIeXVZIamOiMLJwtwRpvVGqorwGdkmprfFFYcsGHJOUHWETPUtKWYvjIUoPFLCvzlqJkbnfsYvLJmjFLRjCNPYnSgzJLMlaiWwyhPtfaQqHTamLNDgTxDAbhkgPefzUGDFZQswBRNnzuZfEIxpHJlgMRfNPbJNfnuuENeZuIPKoMWCqZvImZLskywuchIzOtgnaMZOPNGjZXPDxUWYuFlOzkQcsJXjCjPAsTGvnxjxBxjdHXmVqHVkiObVCHurOfojxIcwphzaofPuKIZBVAIisYeJABbNRjpkDzWsooRgXhMdYFcprZrPdckEapTrbEnwenKHiSnzmjYrYuZUFlBuBJiPTxkVMHOmoLnmcsOGKJmthxxfSJwCJAyDEeepptEQolITahTMzSSjAwxTiJOAollaGzmNwFiitGugEQJwUnlTaPqaYnwuKnrvAMccdiGSIVMkEziXHTkUWOgjwwDcKtdBEggCzDinfaqnMWeOVCwYWwNqcBuNpzbIUPbMWeLHPtqtmXASXIpsAoozqzZfkUpbulSwNrJTEpmXWcaPtyxZmBVPCleyScuRiglMyZCgUYukWlpFNLeDVAnfiRvLVGyBjHGaMAwXfgctKqTkgorqEWxWwYGFIZBBGqkdLWNvmcpFXcIiXLqElfwlpWUwTOSNYaWkqxHczKagqlHMxneMjTcXqYVwopCkuNoJwhIvdhTBCuuzfmnxAfCTzvXopLOqLrAvQGQwaWmiMmVapsoFotDAuMdYExgxIObSDEfQYrZctLgjgQZlvVeYctrUhMebNSDHqpqHnUYmLLlrzvvaSPGzHYtAhmmwBYOdJbaHwLzMVWVFLwIouBWeueJYhUtFTdOvvPSeuFgGhUlOYeMiVcTcFRNhQInSeLVuCCtcXQaTkWRdNelaMDnLFErPEuUvvEKLrabkYlrMBiNzHakPOUJnUJOqAEsGvZekFueopyxXuazOtzSaAQNsvrrXjABxiDFnLEXqgJvCMHMIaEBYgPCvbohEahFniCtZQkaNEDfXFfuYtZANzdGzzaPOjbqmcpufhstqvBOgafyXaFWZDCAmCQeCpnuFMwvdtIWGWDhLDCaHoxbUWfIsRRdPlXluHzjJdMMeLXEhdSxgOXTIgiyeQHZdpObLnYbJFPCSRgRBzuqzsEyTjptHzrFjKakhyxHYLQyjtztzuXUxRsPghARQsEtiLdoJWWplAzSLmGcqZcJRTrWOTRhoxICKGajpHbxbhmsAtnlPTabVipcSAyOSmTvXqOFJgOxjBAKvFWbGsxESNLBHSVZTBxxGXRbIbbpVRoWTtndRWaNBEPwSrcWuomrzzWsvprzgVANUfxpzCzysQVZmaanfRqUuudPnQJeZeeDNtnGvZvMcelcszhhQYfIJYuZJtJAwoxJAUEgZFgFWeVDpABywrfZAOmeZpSiADzweICppzIiogHlWEYzyDCtiWvaOFzcWEJGTOobReGTmrEBYRKLLgkgDTRVyvGhDXUfnCOOKMxqvpmTRygMzsRdHALjquNYcXARblJVvDUbPOzNGwTCtDIPjglYcUvTDKUCobDVZRSrXtgnVhzHSBezrbqWFHxcVEYZNDCVJfqiXAkRFTXGtjuSFVIdMInnTilwWiCrjOjrFdHKdBwhKuzfibxwyZtFLSakDadPEshklOUytMTETCJkCWCgOfrINWlAlPguxnVEvKEZrUjHoLkzvFMBiQdhlMTIQoaSZDXiGLLmyoFFrGttEtLQwtKFdqXKBUOnsLTsMuIIMGwnxEyiYwtjweYMdfrczFijNJlUwHNvtnuQjeevrPIGSvoILjJEEGREHLuxEEKBPRVtuCCZVxvvnIXAjccknpKxUkmwaXitglDrqAXcvcWdUNamZmAkOVaBrGvswbSBhdDLXvQazWzZDPTppZResdKYEciAlrMPGiFmvXHXxLZKjhzeFWXBdQbVRLhKsLZfjJIHUnvWNSZAfdYYMEztOjJXDMmrfvgrbKGVIgajFxNYLscwMeiFVfobNqdXcENRmEitTuiHfKTSNwFCdviIUVpkqhdFaFvqMPgBZcrHOdnZuJVFRNAocTEQporhxSnabsuwtbsRDiWrmJErblDndcQDwGrxkvKsEyyJySXUqjLGlnSDwpqHxyWgGDLtARHyPqPkYRzoROfNINvEayTKUmyDLlSRmwJYuvIJbOeaxQDhpEGqHcczZeSoRMACfskbQDGvzXyykrMvDMSJchPdvvwoKdoLZfixXbOcoZDVzkrIXzOrVVKlJGRNddqUaZiycpKIbfOdatyCmrKflzLpPWEBAxbLpUILjvrTHhjTysRRigSKWYpSARXVSvOivFZmcZPUglELDYuTTkWEyfkkxZbWYbWqKLiGOaSXqbJtsJecAGSyNiNmjgYRMGQstFmfriOpVDimJtNnHXaUjLIdMmKRqhukRFwEbvYsJpgOnZZtetPogMzWomgWbcIUzHDTyHKROfVfqnNBAIoEGzBZKyViXajyeBXFTZtsDMjgkkFjlZwnfZYBzQAVyNtKFrjEwbIYTVjzzcdrrDXUFiSQigvCaOlNAzbEFGcPydrpAPTqMtEJdDKVdvTMGKUotZUIzRCJqrDFuQnlnGUWLBOEPBoNWszHbfgbvlTXrdtSuzYKmwVMbAOdxiJzFHRvIXczXgvvcJMfbQVWShPJDPKQPVnTrLiRrajCwTFhgBKvOTQbpHzuiAsTySRxIurEqQLiqfFDvHwfpuXzvpwCGyaftSUDjKexyItvxOYnxKGmMrRrFDvQJkTrSpTXAGfoYBaYGBegAXbKWJqIXZYuMgMliDhDIlrRliKGzgwDiYCryTniacdMQVKQfLZupBXskHnFADHYGICwYerHJvaRhZVKLsAbNWVMUgMLZYiScftwiPLWQrTShmniWnbhUwWCddnkLHanixPGhyLZJzdUIgwAtelSwRiSvUbCKqxddbiVpncoVNzKugSeCDtLEhjZDuuBrantVCbipjBOAPwVtKRBoETbCSyDrkXyrGIwZoGpJhJkbPLAafLYoLOARscWpHZFIDjtkiJiQjFaFMbAhNpUBOLlEnspTfkWqixmzQDbuZAHkTdvuQlTQgMMsbFkSOalkhFcMOTOczQRScvqJMnEEOvbdkuCNwQlGnFjeTdPHzWldDfBvhmwRoRdBmTwyMEgrQsvSsnPkyaNNNveuyoBWzigwSPxMlEqnSkgFRiRRNWsQxKskdIyroXiBmNYeXgKMAVHsXPBmeWQiAdDzerAzTsuoJXOSbYVsPLiklrNIiQNLascjPHWfqIhjQbXAUoQaSiIfxEgGWMNAeBaVVaqbRsKlyEkwOqQoWleYkFbBxoNMaZINNRTnjplVVOzNLGhxhgVqSGfrpJersoWkSYfdooRWucEjECepoSnpyBBTxQMEVoGWfuKwZDDeoPVOmxKsSMAricSMzhMlpveveuiaQyZTgFoNoymxoMOWcYOyjdYOmpIIqvanbupnllkUVidXcXmcDsfaeCSjnsgBRzBFyCWHwOMIPFELOVFJzLHuaknnPHWjGGCMtWXmqBuUArTQDbFxgaLwBulOLYmVccJGXqtPYbmsfnlZraWpFGABcfSBVgodHSPIFixCHoOHTMdsvEjgdyKIkxZLXBMuCYNekZkJlbQsOLCsokQGEGejKMuqWGnmgsOoiibOqLPzSzyZYimqiTnOGxgkxKveYZxLJYytZQwXoFAPEobHlhYYDdQNjsEBCLZUcVZlDAmFeJfGsqBsbhaUmLiqambJbRFENdFRWxrYbyeuIsZKFadvhyciOXbHeMkGkAAQgfEAADcYWKwPIdsbigWUUSPZNnqfQUODJjXCROySoaCTJEGDlgLoAmDwBgjnqPTLToqCqErpOovHbnuPTKbfoqPPDOZEWqtvDehVwYtvzFAhsTWGsluLTdWzalpXujyUzaUqviiMUcfkoPpaVPyXhsIhpRzbWRGjTdwFOFCTAcqzBIzrORhTRdndHVqIKWaBCOZVDEijVXIYfHpRmuRNeWPMnDePWLkKOlGvzKwoaUrvykFPyHfVAeYUHcKAPaicSIElGknCrWFjHDtaFMSaCXbsPBmpkenKRsIHhLngIeoAEUbhGtYGgRwzdbYNjaYsZLDwDhEiJUdpiKnWNiciyIUYEjaOevIseZnKdDpXDDAPLUDWXWzAPLzizFMCZVpzXLMnreUYWhKChYiSMthPQDMlOhppDlitJkOGliCReNFrHeFxaSyQfjHJqCPzIhPkIXiTsMoToEctAspGeqYdSjPhZIXcZkPZiVCagQfUPRHlGJyXvelviibyLXrXliUgwdWyiBSQHJyApVmImgrgFywuWwxGxiQWEDlBfWHkVinqcStoYvstCNFdwvwwxPmHVmsUhpJuwybRIFsMqpMDxEKPMsAhiRQtkqZmnEkEKgMiWCYUwFzAMmrtvfYvfOcbRPUSRySKXLaTjbTPZOozzvQXsmrWazVSmaPffcLKFlVWDBrIrkxeLQduAQqUNiRauiDqGShuONgTVqduOtuDwNxrRoOHqKcAfXVBOdGvpOXXLsCWkBARYQwjwrwsqxSuDWjJaAyDWvEYkpEMoZEaAcWEIiGKxKlPSVJhBiRkrCSLODVGkIgFUiEWhyBWMzmkMvNRjzfsosCRGeJwirbdIbepRqRxdCeZbcbhoiJhTIbbgFoGmhjxfkZALNDhACBkdrsydPxwpgxLULhGnQePRAojcQXRlHqLoZGYNDrlvrcNLEzYWeqZyKggraiybsOXSuGxgpXQcNuXBKwjdWqIeftnqRYBjPllcLzHWSSjuUlTDpIMLxGLfYybEsuByIeMmrhuVGiKCuRTnLQtZisEEBYkRUfnflUgcEjzbgcVGODIFDPIaqqnuvUlaNvdkiTdqbILAJxAYbCdWpdSkQEdEoFrsSUEQRppEUltNxADoAJWUWNOsFxBEGwDzEzfSDziZAjWPQVicnGRaOVOVBLKtnqfKpBhzLWtXRIgGzsFhDujeotMXgvqMLxbHJrIXOLNjXtxIYmZsAxwxtrQSZVcHiEMoxlTlwaPjtTsQPGvEdjNURBzzfdEnDEOGWMQjFjxyPMPcpJkxzxJhQtKJCdTfOzyffZlpwPpSAlzxddoqVnuwfMYwDjROzMWqvXpMyesaUfDkfLgmEtYpsrVGwqoAuuUlfaRLQUmtVIUjJZRCPlvBUOkzHGfjVHgftUxLjNTfrSEDUTmIxChefZjcpiSfbXGpkFZKUrlhYbRjOKOKiZVIrFKQjRAYSGexIBraTjBwyHAvcmskUdYSTDeOulEmNYyiVuDNKRrzSXpNJGFRdZoGdSdXAYiqZgUDHxglnwTVZIYceePHXXlOrPrODFEOHxgFSLfowepOPazoNMJFcpwQZzAMWWGoQwTquvfVqWAJxYriWOqbVNnpRbsMYgALPwRvWzswMNVlPNIvctdXbwlpnmMBUGDanArpclkWcNWvJaSZlpJeDSQDEadFdykOVZWrOWlcYgeIcNTYuLnPqeClOYQaZDQxTSSJCteLlWeEGJzWjvqFHcgwGVJVTOpSywOOHhswWRMZYvPQCPWlMfvprudYRnGTuPzHexRXHmImnzfXzPdphafcMcSODwQTHginwesHZaNkomYVJiRxHCBfstqjxgiMjOQYwdDBbyeaJfCYOztOICHjupUzKBfxJRsyNkjOaSywWEtjomuQdnxbMDwxQwLXoSDnQmnOxHJHZQDAfiwLuqJkUBcxZKQwvvjtIhOTnnFYpwMifMgGDiwysHTQmSvEaMZuCayJpYNFfQfFfVESRukfFYWaCgWxpbzDhWzewDmKBPqQexCKluykkXULskdImBnTBIxpiAferKeGxfZASeMenswcovSsJOpVvhTtpNTQKXjfZTWzFHlmdxePnRsRKOdrgkAbicGmLUqDbYoGFSYxbyzsABRbckotIVkfUkLBGeTwCnopgAFKsDKpWYhnpfcuvVITUFLgTrDZnSiXLnrNyEsKZjycHJOeBsahszugZzEPoFLzyydQNCDlAlkvTweTZWxyDOzOTOqSwwCFuUBJFADBcGcvcXmhAcgnVeBJEqdtEJIHfamHBSHAxQHqZwbkwHuadoBLIxejrFiqQtxgcCZpeHdeescjyQJvjWUutKZAOHCYhpdjlUdrnjiIDfSZIFHPleGMCmlvEpctjPaUUMMSUbdcubkECGXQkHqLNfvtMKisbORcrkAyEUNXwETQiCYthlisdpFgvdBPqgGEzwhMncfGNEUqUeylqeisyRDzUNffzDUPVbEkjBGWqQghNZBumWbWhVyBntXiYjAmliWrzHfVhKdKxJPXQDlXUadbowHmKYmZwxWsISJKkMbmMMBpQFeRatVODXPCXOAFFYeNUpcuiMLNWzAIEptVFHmkUEpGOJGWnacgrnzflazfDHuKrWPytzPddeVCsELRWXCardBDdGkvcsUuXTwHJknbuggygarLaRiZUsxnsAtMmmmJIitKwSJAfzqzquDBMhleaclacGOHqURGPfcbzhjPsaeYEEWKJKiLfrBhAGzxeSoFRkPSZANTBixmLobEZNpZOImTOiGZJgBcWOMyFHbFrsyYQjNLIzgZOSEPvWCUpGUJYDaefhYjCSXWlbDGdgiYYQfSAhKNKVhuwVuIRLZjuMKEXvGulqokyjuwQArOYiUZKrnTECONYycJeUorHfqyQxeKtYQoHwTyzeGgTpDrbIJCUZInyebBBeRBvXgjpvKBfxbeQVCIBBlNgUJePzfxiKdUzKAjrBWjlBtQOaJuUTkyIKxzuDLhLKCCmKGEHkrQPKWLfFozYWdKSYUeIWAUJZTWbKDSKDysxHnlPXhhQuBeIyEdVsmXgvnIrAxFBrPpRzhfHrzhPUrfMZnKvutsVNOLQfmFqXXUmoVcVXoTqxZkxzOcptGIfrcxloyuHsKCrsRKalqHGQPmvheVqBHLmqJufoDtpSsiGQFfUhaRbfPSPIOxMGsKmLXnBOLcEBhBCzGpxvtZCvwpaYdGWlzKwSDxqrWGCWcfYtFJuhsByYSgqeZFcksMHCGYrEkKuxOvQHwXiEGkFfVjQkOuiKCUiGaCAfDTjzTClUGSYBiAjVgbaYLRSvsJtKDijOrUxYZsjdhpzgMSAXkjOrUUwJMWbxTdWXARNWnTugjCJsFietPYTqTxQRZVggDKATcWbAUmrbcAwyUMoZBEUhvinBpyjVXeZBuNyiyXnNhkemFXexUIVtUkWBLGSoTiChMzoLxaLHQFmiQTGexUCoYFSZqhDQHhmpRjkdQOeEZYVNsPbGjbMjoNPnzeJMmBLThqhizuoFrvkWKPNvtfxvRKALNjsUZrxujRASpYgbQIxdDoPHiDYvuTLCoRSRVJFVUpqUDjjTBAjvRcJCVKQnAlDQEDYHHhrcnzXSaGuSJgVtWiOSQsqPOACSIktQLFEjlXdDYeIFFfRGuEqdOyseMXSDkKanQqtDuEQSfixxkPWzjSEyAaJRjOKIytHsBVyADvnUTXLRBwSwFsMyOfGyhcgnkQrixQQJddWYRzYoiPmnuxhYZlwyfsFUQWaoamtzvxtFzQRUpWNcSMjYjUDqcTdZwFMijCVyurjrVBqxPwOndOHNYhUYFZKYOmPuxnbtxjaZNxXXzSaXDeRWLOvuLQUZWsEcLlRJmIZtHpKoZVufpMOCTCauZUaKhqRTcKIeJjlJdNaEldMsrBCtlgvzKAKOFflbLFieSjaaAghAcssgxbzoyHCOtndCQxZYHNMneJamVBsEZIlFCBrGHyBIwTtZgZrnBWHbEJEMOPBvUtNGVkzrnCVLZIpZoxNIbOENZQvYJzTDuHextXJWHWedvQqoPAzaXKHlkIKIxpUtQbMhZPYPgQfgISEwIetsGHsgkefUWvCdLMwYZUKzrqUoZHTbKbyxIJhiJljEUbgfjBYrBbUXyFlTFvjrBFsjwnyOLHhvUTzLLPXdjArZylwamzmFYZXQblCbAJeyBlKNNLGcbLfpxSCkUQTuLqzYYztitLjABpNrPFJBoVbmxTjwJbgpNndqYMMfwwRCboqoIeGHGltedrdULEQmMRxPicNiigmBVjlcNtOGFfOWNGEeKmpzGIvxYXFzdIyWyDivkBnKmXGplSrbdTxGCKjVAOnLoPZzSlQuiqlefSCgvWPVUYfbuLqcUTYftqzZCYyRPHThOSaDvMpMuUMGjChMXIqHBzWNLPDsNPAHMKqYJynpkdMYRcogwisbOpeyilxbFzCwrDocwPCbMowMwTqCjtuYNUqQXFoobpCMDqrDGjgCyBsmVHoeGfslpUwFKqJeKhUEIcbRXHbSMaUuMzkTOugiyJXzSTGhkXAhynHTYIJODsCWxHCXDqvsWjXvFbaXzHJpQuXXnxNVDbUGOHIkEhJiWUSAgQucUlKxAzirADDEpCKiCtvLVRUCQfPjtbFCktGUJOdOdOhzBtdqISFLAhfQHRgVAdPRxnQYouoSSzlEmgOsuRLBJQsixGNWxLaZvVDbYrxrCeZtVXeZklqUcnzKgtIlXFGQMLHrSErkTfaPUpXgfKznkoHvdhplaudGBfiXicgziPWzOVPIWSUDaKMuVgPKmwEKVqdFUbDjwyDsVsHNrJNBTtudWhaecvZgKbnNVPSeUUcbzdSTmQkDjmULusuluUqHJpRFTFbLxpZWIjTpjgIQmSZIKsCoWefoKRFVNlUOQzassiNqhwnEJNOeiKSFGCqbKksmAXHkbeliPzJDCjrGZYyAJaQhfdjSwAKczMxgxQUjVoJMCcGXJYkoyFJangpXHolRmeLkTgrZleSWfrVDcjjXMYojUxqCLAPTTWCVdZkQpCaMGoBDJEVuuBGYWhJzfknhmcMFvgsmvNRsirXIYDtTmPiEnxEpMWgmZTAdlRffjZHRtFuxMNXtSpRZTnFTWhlAGODIXirsrPywZAfNvgmMLGxvOowSQHGPLXZIbVABnptWYZQyotQLLQVETrngkNgRTmLApEmLfcustNiLxyUbvdvVwytrdLmgNHINtWOrYJUNTNZunNgNuixTczAEEjINBbiupUuAIVHDIvuAfzpXeJoksoXDCyhpVrfAmidLtGwRSOGUVFaoYqztOzsqNZLwRBBHZAOApsMWTzWerEnDEDzqcoLQvykAkhswMGRHqzapUexjJKmugOrwMIotAATEtzoBmsSFRwEiZBqgWVDEEXfENGCvFVXTDtCEfVVWvFNNOmAHymRhPCNgatHIEoOPgsulNZNYiyUDTQnarQrAJLvKIADAvoJvAfbfFIxXCoxpvmflTxbGdhxqWJrdWdokPraapZxtlqQXccsYbvpcvnzWKBuXFyEyTRHTMlxpQaKJtoZCYoezQoYSgAIgiWxaoTOfQXJcEgFMSpdeoBVNwQmKcyoVYEMTifjNqzMVgZLrRkkSPDtxKoNYHhvNaHAxLrKvmWEDTqZJYyyqcHGyryOcwmizGdSUtjRYyRAJaHggGPjHyQHcJHNQdrjiDtVplYBWIMQeSORfENUMRezJAgzClhLORfVTUVPBnwMCtTKOwltjklfGkpYsrGJyevNFCNxqXWqSxcCitqpFtUWlQgFLtYCeABPkeBlmRKRFfvnpKhfhaZeMRngBjyZotYewETnpPdVyEXEUHlmGDctQdtviyDNAdRdNmhMKHOlpGWrPapSNDlxlCtgWpdRzIPDvkDauTwuFFlPQPriqRZRPRbIzcqIxvAKBnxbBjjTPUpkSSmkIZtZCknLiDZNMUsrsUIyoTCykziiCAKXUeqHviQekQuSRbGTnaQCAAvXniMexvFKJYeeycYLtjrsyTDmUxskXiPtwebaHpnJUggXXOStwRoMbOJmsNQAfjTeZsNJWDHYxbiHocVBwMSMzWyGvbflcjODGJTFHlZpjKTcOgACJGMbWkifHgosXNnAXAaDTjqzRfJYvODvVWTeXreWHMayKPcMDXJIWCvgdjdVFhgYiPUWuXNAAQeXhtlWcrtGoAGjyDDDPaJvQtUutpojgrIPdRTCakgFIymhzgmIrOAkOnqPjBTGjlqcGmRhGtsLZqIToQtrZEbhYFTxqwINIlqtLifReINjDdwbGYuumYbuBARyhVzQiDiCUKkgpmNyUyFgEwhewOeyapWZDHiFdeSncHDLlURnfGyjIFeTYLCTVxuVoxpHKgxRgizbhPzSwNouHhZJNbBmIOYyDeAasqqHIigPCyWoTtwGtlRemWnuOgTNiOcnwHeqRTPMzJuPMSNLvAWCPHJvuyosHlDdQegJLPlmWrUmQNJKCyLtUGdhBBcEjVagPGVECUhjNJXgTdMfRopbRwbwJwttsKRXSunlMtyrYHlzfUJCLyGteZbYieYPAtOflVvCeQbrHfwzsrEOpCwgkVUfAdyhUIreWjnjxNYgQabMtYMfRIhFsxfxWhvDacxZgewRhpspFzPXRENsjOPSNJYyaHmBbIkQWSEHdyRNQYoVwksVuJFqNBGCvbQqzkyrYiJBUXuGlfCnEEaevrVfVVCggSkGLFkdCCgNMLkbPCxbjYrYDTQsZjMjXCVSwmJsPHMagHLLhfIVmJoGPtmOhdWgonAcCUIedXVlorslMZFCOVjQyovHXMjMrsBsFVOBuLtPRrVmlbayvwoqfhmEDgVkERrozxUKtgUkwHBeeyuqqBlVkLHlwqAqiQLUAfGclVCyTNQoDwlhxqQqhXhPyfzHyEuMXRcMFWgvGXzLpehvDrpoTPiLfgjembEtlxPNvmfvlKSvHBPqqcXQoiXZIImDPZyMKRQKlhQvZaQdmXlIFXCNwcRbTYyUPEZGVyJsYXJBwJkEbXJxGAwfxhAxcRLeccFnxOhooYlgMwMRrDAxFJEnUaCAuSnjDkyVwHrGOOuIZFklEHSDpfHZPuXbEWSfJZNubfjWQbMnFsicOHgLfuEbswrySkehvtBtxSWEKeHBrCjzugTiJzGCWYFPNoWeYeoSuuEvJRJoEtYMVemZHqpVOgJTQeiPFcSBnnBGAVMqJwqmnxHUNRqFUaqztmzjNhhmwlkFWsQzLdvfeFCtOOFmdJmvcmGftedLUdamaNRvYWgTiWCWMPuyryqrntnfakNaTFgKrspTyMAgskyOibldyrALxSmxYGqNUvinQTsVVbZrLmVyJqZfbWLMeLRSqkgFDhmJaoccKVzGTwXUlrJkdcHZEhRHcoHcrnFOgjjKUQGwAeRwGVKPNmqIGyneFLDiTsrDxGbEWWDkbaTVKxdaNuYZFgKltFWCNTWPVbfAZTcJbpnIDBPqYcQujxjiOEBbaBwdiensAmgLXeZcgAApGiZFziEFCVUBPautdgVaxLrwsGoAIQfzMNOAtNQnsLSYeaOYqJTbXVhAXkHgQZrTsEnSMYIgNoKPbMvIqfOHqJtjcaIoEPofSkfOcBKCbBUTUxroHNSuLdXTdjXoSvxPokoCOCggavsDaMUkAoyhwGifACywbaaqreGyGdyXHWYkFGgIIvtjJAHXlPMceNpqSpAZOfiBNTuluGEULpjCpefGhvCwqesrAESLMRSSzCyKNxKNSVmgkcmwTueYHdOFDGtluGWVSsVCXopMkTonqehtTMEAXhGBzkJgQrwHaOROajPwqSnjNbBFCAcIRFUnAEyRKDIJZVrxEEbsslutqkANthbWPCzZFLxJCeLaDZVUDufFXarCdZhlcuKEWAzKsWrefoFplWxqUbvEniMLXVVmjlBtoUdeRdiNlLGOvpRsYumdrPClIsLPiTqSauBwuyouAoaMBgDCtJYNUSsvwAEhFOwyQujPTjLXtHgrohfuZNOrweQhKtffFIsfWGJeWcZLFqFMNAGyRjTizknmHIiJTIBBIxCxNXmigsXWTUAChGwZfGryFuuDMHabdpssEePjxhDHoRbtfSiFwcFRneUWnJyFzGmVhpkFeWrNecEyjavRssmelXfaZbMTijhxzLLMbluOidYdaJVoHeQvMDcLQtzgikgMUtrMhTfkEcrOeoRgMRICWjXGRuaXFZqwYptwrdUlgPFBkPKWIzjCPinYfJeDJHiVlvHuJxFceqCOmnBNRBpgCfQTQCKhhHDFhtLrDIKVKiDcvRcHtkIgRdeDekjCtirlvHaBgqhgBKoanyollbzxnkgDxkaXWyPDMJKRhqUezpakZWFzAIqReYSjfnNDaZTjDQrsloPLoPePLBnMzpPDWpJoAAgeNlltzeuxWkfehhlNSdeKUbtwyGognDPfSynSnSlliSBlbKyCRrkmIVFptxXgjzTPLaeaWftSsWELLmhHLahwWBBFXmjoYMXgwZDXFhqWpGgyrBFfSCANpIBbhZhyEQyzBdngKPbPliDOzxpNchzUzZZbwwqbvdodryTATrriyyuttIOBHFombthsvZnuOuWBgTWKLRePKpLzNpoPkOvfXACCHINCJPxmikamHFEeqGnKElvolpPrHlTlMHECGrucbqfRlfXUOBnmGmPfumbLUAjagnPDgxfhDyFTlUpsvvixUPZFOSQGSubUsJhgQJArnmGKgALkRUVtINPMiljaMCDtTqYFrAXfygAJgWQERGHkBRAKvTRSukbGJAlHFLWPeDGsNDkFclWyANWgYprTRyeTQwWpZbpVHOvKqNVDixzjsNAHDeMPbcGPsRYMBHSrQmBARJPutcdxEdsoLxWwZVVCESjiOWJqjZSPyVaSRxwgypNBuzkwCIsXfGqydZwwGjqmQnKBPdTtpPvhIfoAMzvgdiOGymjpOtEVqOEKmLSpMQptZRpmJnyBAfTYLsxOIQcJuRDUwSkYOqYygrOhERQkLeBgiSnAezFSuNmVJEJnsLmDuPdETUgWtvoySGPDAZHRevSXPbyqipXTBmaKvGoZOYJaplyqjFQpCaTJPoaCxvGAMFzURFNxnkIxnKeFQFYSIcxPpQNeSkwZJjMQTXIPLxmqbmjUMzXvDkPwWERpTLHKbltmwQdYWrRnJQFiLeIWMMsoOJHgsDUgaUcxHEyFnOkpXQBGurRnZuJkhCCppAVyOHVxnhcsXgQBysysFDCBYMOaVliVhyUmGLBExjQSUkfHewazUeveEudYOmuFoOTiVHIAkgduQxeVvFNTEpBzdTwDRypADwYFODxiLnhpTgrPUeziecyWpPGCkhQaAMnBiQPbcdzfoltPNIVqBJLvNNBAIvJYdEhKvGMTTjhZqtLykIvtAPAEfZlmdZzJZsqvmHaZuFPTOOPNIQeZiLGJbnlTExfyvNXUvGTBVTuxJyLDYAMqNZRwWehRFPZfrNkdcODtLDOxpEQfXAVrqIQJUUHeYWMjlQeIsWTSbliCvyUnbjgdCzDKukvIuAwMeVdsPrcaasbYgarBcnNoSHXVgkHncLkzgRUGboWvXvxhscsIBuPsOlyTYUAkeffweiqndOXlUtcqkjsLTSpvoqZYnSYPJHsYkaTNoucbGwIBOzaTKroEdDyMHUyQQchnfVCZlkoPubOjJwRWsKwhaQzcgVoHNPdDtDGKeLuQgLLUVqOruMUiEHPcHGXALcVilJiXzFCQlBftGRdBzvZfKyhmChKsvKarXoQPpCxhYHnJbLHojfcVFVDJDdvrBBMkmZuBEklRSwrSJEEGMRwaRehpwmDnAHoHMvmaFPpIRbmIXoOHjMzbpCbxvEzCowkXSwmMcswuaUQlKvXjWyeCxEogfySmXSJefDCXCNijzzXUCpXSMFNkhycrpWqphTIHOkpoQNNAwGPDWOCVVmVjLavyZuYzzWvaqIilxdtnZrjKbBHkLhSXRnhVuWddhiJohqJuPGStrTIDsbydGOPJXVLyuROmbJHXHNRxBPllAWSkRMXkGTxbXdVZLoVuTeYNZeOgdGAxYgQKRjCoFJHHLdaJQgZPhxNMBmWWXGsLppHdukgURoAcxDUIqkDLfKuxkoPVklrdleARaXsLVWbRRFZaAyyBfABAPHPUWFCnQZhAVrvjWSZEcWiXEBkZHHIuHhBgEezCurvncptnvmlHYThmIrUGKFvqoCgBCtvwjuLQnZTbIzLPHlhrEJsJwoPwtuPIstXQdgsHQnuFuufHSmRGZFcpCDenNlPYQAhwhJAXaCbSkDqwmNVAnjKhQmSQTnQhQuKcnUTEaviopUgcmiCuUVOmUsxUHMivJZncsYLeCNmUzPGaJbaJGAdQMmlbaAjBJYWVXSWAnKWYmUhHdSyUWNThNVtODUtJpMsZnSCHwcGcPMXPugciSQjpeGmhPAFDsOiVwweTWGQdOjMFPEzXaJCmqYSHBOdEMISQVLqVNIYjKDLnkTwelofgzJxnMqUHWVQmaIqVpTJumAlDOPeEzNTHTkFqnUkTsRjKGgfbWauJjaXeaLKurJtXQXzgITTeIpizDSkASBpXrNQfPQhQoVVXzlTBmNpQMlJVRTDdhottFwWdpuHTwKcxAfCFZNxUnfJahGGIdoEYzVmncNDimFlfwzCTbUYBTPivTLLudCkpGhdupqjKHvvjecpXelwMcmRGXDJypTgCvQcZSBjITOfNxtNknizsWxByyiujKcKgvPsAbQXkAizlkwFQcDbmyNOlUkWsOnzPgKlZMbkbHawOZMZCKNFSthEYKETJcPhJEhJPKWHjMHntSAaYedMhJqRtWUhVEUpSDMlOLUNMbMXSHuTROiWQFjyfYwsqfqfpKlvTVeXjGxCGDCgdUhmPJvUaMglozGWmRUqoxMSbeBAUohkWKAScOjZlhneGkGCSUqLiQSotqphkyCyDkMmDnurjwvgAfbzOvHwNrmzRZuEmmmpWZEsFEVNJmzgmGksJDftddtcYHaddLqGmyFaFjGWsOPDrkHGMuvGxrQYvUSvjYqoqrlfUsSmbTgsDEBwoNpkSOfgIkChNIjWTxETjdIRMqXYEnaptEBvbYSsasfVfzVHBOmbPBKqPvyECwuhdXuaGuJjFSSWdmZPpritIzahNQADnfeALjPKnVzBLUIBFcVONSEbZqmpidealeskYZVvNkaWEdreIrfvIAZZIYMrQuJfnGJdbpkxSCzeZFUQDBDJdApSxYfcrbVeoakWPUaaCRTCkmdBrRonjYFVaXyQkMXNCYUViPoNyeAPWXyEsvsbNrmQJKUHtfGvTvMUlxEZDDztdydwZXdYmCRTwpmpZBokHeStYNYNiUmpbFRWNgfvOXuuxlkpiLAKflziGzkcwtAPabnJvPmnhPElHQMJDYBzyENfFMgcMNyToYTEoZKuUfFmZxdGDrTBzWgiQIUmoasBTjZZsnHCIdrNNtCPMzXMLfWnFKlcIXwCQfLqjXyBVEYWxOAQtbXcKVEvekbrxcPyMWrlmMLEdWqknGfvcpmQpUAkHtDokItyJaibYLICWKEIMtiuABqgbAeHcQQMaQplaUhtLyLScjGFFFInkUyndgoyuQAflkauYFcHKsXnrlmvBIhFjQOvXGpaikAIuhlqmERaUDEmdFxwMBKBOuszeTJziKOIdUPpRJemPNaYJEPZXPkTirfuTJGpJGuJOhYRtgONCpucqJtQgXDuzwqgXRONlSnNeGiFNlhILvGjjnScMRpPDsmeNYflZaMjnnSDeForwPjIKmnpHrSsGpCTScVeoIezsCApwlgaclpmfCrwHFJxypnOpGCADCxjsLNXpOsSezGGOZtEUfHcnLXlELfLgeBpsAjBzQJPDYBOYHJCVVECJfLXkCNuEcgXwDWweEWemFcTHMCqNLtvjWQWRJtzUjhQITaiLchCvEkUDQyvlwwcZeNEmRpJniSXWRtLQRSNdQojEKfVHYjTFgwzkQnoCSqHsoHwKbYprlsIPHAfeGvlFdMPBCssciyUBEbeqoHMRpxPqPCmuYWhPBBjGQlCAVFiQkmaxwvOjvqGKjAkTrZPdmnAWXFBcIROugIxsEshavGNxwlHJmSPTmfukQmMLVpSnsWSlEHkSfzFtBKTJhefRTzshxpSDyXZQJaIPHEJeISZQuxLKLFNdzeARKJzXLFgxHfzFlfzYrtOEVEeBejaIDApzLzhbigOZVjAMLnYAXEoDoxZfhVCDtUpdMAIqTczKuyvkpsEHXUaRqexjexblshCOoAZQeoKmEYkMCfAtkNbqgvEiIXbTXjMLqgGxqKrvuYynEjYAseaCGJHGLRYAQgxocRUkouFnixVSHzQvnAWMeaEWrfqwZUvZMOrIsuheCHmKZQxcNEHWfUFZXboFbGFKVkzfSoBuoeljkDCgOiYifXpBdDiAWmhKPUFxfnhnLkhtexKbuSKcJEpLmIjwxXAVTAtWZXPKLCfbTQscWgrwSapIsgLJWJXdhzpUYYOOJGZeYRFkffIoBrUWXPKXPGiWoXnVdZdWuliytMmHNzrzPmfEgZJGxOsVYMvBWckRVnkcbNtGSxXHVQoqRBcQfEBNeNjQNtIkSZNJuqjPykLlhigSFATyTLFQeqmzaPJgbPHYpqDLNOziJcwCmKOqfefGCCwERjQjWvglawsCNoHehwVUaazHSwQEqJuLrThGxJXGudfVqbjofEULalsKTkVxlVoinXsrOJIrhPjSiEHJPXuEJdzHWqbXIprcQRWXrhxwceDycxSqpNfhjexeanazPSGJGCcNwdYnIIYoDTECboxOiC</t>
+  </si>
+  <si>
+    <t>ZuFwYwzUJqWgVnmMJokxyvVTxfDPBXVNKCEUMNwtgsbcWMNNPJtMGWkeQMRwByRmJfTyIqNIhqAjZDHDhJOYfSJMMTYDQKCCakNsCzUoaacjrEiNzyvAaDkccbNGmWFWAiOrdBwywtwCchVoNCXXIyPYBLZwhKXMdGHrTWRuIZkQCJvlAqxTWXtzohhREHoWHOGFjOBEykzAqSeDPFKQlRvqbwUhLCFfBnHYCLhBNffpuWGtvLvXjSkBeCAQxsQBvyRDUYZwPVSgIstcTlQvnkzLeFNhkIZLfmXGUMjsfQoTLgrIcbcHqmNkYdcTRxoaNdmcZVVnFeRXwAVWbTMmVjEbyxBPCGemGcuAGsbbRtoGOzEbtMzOKNkpEBGEjMZcqdWPtOfkhLqXzIhqRaiYgLrYcBputISnspCLqWAFipjfYbbwmFoRimDLSuiGrXGhcncSTEWDDnOiNjMSVyVfyIQMkilukBHoaPEPnMyrWRoXSKqVopdwicZLRWqXGDlNQSgJOUjMnTVfthzFToEqbjaaRPjfqLRckaYqeIoeKlotPjGuhGnuwfsLXIAfPszGrdNHHHFLpPSOHaYkKwhEmdTfaTTvBaOIhzKCVMSoWhztilpamYVzVAvlCPPDfjycolweLFSvVnZUSwwTuvwIOeIdNuLgydCnbqmoYnryGTyXgTAAZkMoJVfLJUQckGcHuhxKDOaAYUpnJEfmQNmItlmyDxhyqfybUgUsKebRqwgKsfRMEqJvTbGzsZRgSchpvxMQeILXwkTHCYiQXDUJhPbWjeykcKognfsEmeGuRSNXgwGvNxAifiEKiDIoWgnvejsUIkgyfdiaBNytVZJZWsCnaKWFMrIQeMYiFEENzpoVqmoRzCYDatZHTaxvNAyGaQjdMKuJWwjsmTuBZilQKnuZSHZvmAnTNtfhmMzgmmtaTWGfGRgYeSdXUjxzydCeqIIXrYqtMVAlGfCxWQMelDBXocqMKhAAtyExeCmRjPAyyFjwfhPwxpCwCmXjDkSmjpqYyASoFzcAjerguIwlRkgPdlDbpSlfYYeNybOvYKtuIPvQWfGXHuVFFEuiEqJhuQNHIAxRHgmkrlGbAsMmSiTCvNwENqqeyoToyRWhCPcunhjGQKvGYNlCrQbAPWWcRIdSeZUaLpAPtNBwJZTlxMPyQcoxmifEzUyymWHvmPvcMwWEhUXhYaJAdukVfCFHbpGtkZPNTZCmszxaXoUhWyaLXRQfPMRNZMxxgeZamEklsneTvwthtDMiENVcbRdHHMPeLueikAwySesDCaDIuLOWqcRRziqsXsiYbfJWPJLHowgKuzPYtqIHWqlZumlVAeGNOZuVgdGDnxnKWUatabefdvFRSXLsHhRjXxSnapRPTwWOGMFacfuWOXznvnLBTTSJBochfVHOySKAhvRxGrNGAHyvcGAEEJUkvBKkbpWpqELYFhOqpJHkQtXTnJbckCLhlLqiqlyYlboNOkWvWuDPNDGoBVhlHikoQxFZfIMdgvdVofzdBATqKyUPtFFTlrusUJzOWNLoTLiymWKIjIsdhumftjHsCkRawTIPJrbGTUNPiVRhpiiCaAEeFALHrzjPbgMIXdNCfZYiOYxNCxWjKjnmsDvOhvnINdrthWfdlHaGhtcDjcjqzSDoWrcdylXvAbawmULSrIOShRMpyeIAWMqTmmZmRMIQFAweIWTwpDMyIhKBoTWgtHOSgdNgeTWdoswJxsrkSPmgwCsZwGEJlIpQUlqLnEIRUXkmgRfQPXeLVhqMwuqKyPbIMmiLWlbbMdwociQqdwzdOBxSCQyCRYMTjJvnjHIAvTWkksmuRiEnmVSmwMVkcICVJiggPNwcsVWBekRyUdAYIjzMBkvCTgPPRnivSbPgdCqtlGgVUOaqchZRfLwzDlsMwqhpvdNTQBXdNWqgLblymPBofVtmitSSpHmVlveKGYpDLlZUssltAxKfdYHpYGqeCilHsSPhCRDxUOWKHwTSoMyLeUgXUtiDqthwlFMpbeMUGFFxoAcUaODbnSOZWHIJXPMpIsmTJKfAqrlyYthbYLPvFWkqywUIJGAnZzGdFchtNZnbEookhSZRSHPYiGlditfCzOyQbDbVzbBHvWJkWlipPQkhjcyGzxcHMIoiSiJTHIlNICnTWKJffhtWlmypmENVuTKYWLrGLhutWdDovQxFXtJPjiIdTlPwfSoXfeVxrbKgYPZwqauwFMuiKooYVMfHjRmcZEEyMGtSyAXzISqjgrgneDgWwlJxAGjiqwStSYGaxeKtnKYqKqqwjcMqlKxZHRRiViajHyifcwLAAdFDYROMiiNtIsveBtKUGFWAYmPfxGvtAANIwllnNUPUuxMehilVFGgDYEFRxMIliseQaLBzKUpsbejjdXyavWeFqeMOozrVWxDDtqQIfKEOAUGtMhurkNdPGsqFeBPvnqHQqOVhZmrOwnqKaAiLZkLwSfuiYgcEeQIYzhSbjgrlUFzOztgkwzQeHUNebbxLAGquRDwjEZTWOGoxyIDOfYSAXKOIWImHwXGnVVQaXJvRxCDVeONRvLwXKUQvRbsUCdpkCLoOOuAhKcILBQFNlYvWWHzxudgCdptAaLUsSQFkTtnPxkpyypHSXCPSqpYdNzJEHjtEzlvedHQeNACjeiWpysslJcLticTXtzFtIckFigcPaYWJMIWCdDGrJAFIWvTVoVgfmRcfKsRVCWZZVwTnPbayZrVtkgAuspYlhhUXPNODpjnoazYCtreGGoECIDJpRMjvxwcgZFCyQuVpKPHLyUGtuPcFoCDwEqWXiGijpBgPAcNtaNNoLVEyhXGsuDQBjSHMoVhitgIZIDNfpfYDMEqazjIeNWMklMADIyabomBpoAWnjDrrmKlJpcsirnpJNihakYPzTSLRFYbTPYwUvgPjnzahASzDMIDncdkspLXOeYvsXzaxZpLZlgPVYhCWlQoJMAukGHOHrrrtoUYPPlhIJIPQMnwKFCHeRKaLqzEGcsOAKxuwvgBfrHUGhlJvDYoqEBYcpVVfElslNQUXYUiqXfDRPpgHcEoZoYMVWQojdUitTgBRFkCARdQBgymvlRchgIEfYCWYEVaaghDDdybwOuOxYswGUPmHGfHnUPMvolTnXGDIZoUFJYTbeCiBhNUiBBBYSCwazhdOgpIlVgzsjxfmYhgZFfKhPrwgQusmPQLWqTZPxhiXDWKFWgAuPEvigcdfGiwlxMGVuTBdukIRlTvArEGbEceDLhbxfCZvvYudCedIUfrzJGsQnQHwwKpnisXXmLicSchaimKhfGfsLaBlWsaquhPcDAqeKvLZbJiZsMkmcjoWyjyiWlJUxiAZECMFgepqbjaotmOvqOjaWxNygjHnQuezNKUbUhQdZrbbofrUATanHjxwApctjARBGRlFIgmLwBtKGNVvEKkzrCudNWtVERIznmuBXrWkoHWxrkERFFXjXlgbcpKizigIyCRavRcWeSCHiCnnBLIlIzotQpKRadPzRKEkfzxpFmAFpPHpMhgILMfezbulCppJZedaZewhxnRhsgBjdIZFRdllZdoxsAnCFipyOqQVCTxdZSjbofcyhriFqnPKPJwjjVOUEMzeLXVNUbxFunYMxlKZVAQKMzzBIQHxvfNhvbGcrZqYaOVJcOEQrYdtbUKiqAMGktLaKHleGuEElhjIIGBydqVcjoNIrTlcQNaoOZMgdFthSlHNCHxAARdRCTEEByqGqHxYuVMZXahRnOQaRbcEzWuNiLCVtlnrfuyDNVSkejsTHcxTvyIkpJMJWRgZlavVuggdcxfDEqkGwpXIIeYSCfkMlSxxNxlXAKBALmQZzLDyZRnrYIPDCypBkHmnXGPJLghIFMLFexdhjWgYiJtXqrgUbwMIxiMvEfFIKuyIpCswyeyQvnzUtHJtaPPRfkImMwMCgXQofSeuIAqkoidVFdErdmoTbctvCMfYbqVEEDVHtJTFzmEaJQVrQLKUaDYPNXfauBkFzoOSomippWpQtDucEdCkwQdlOTHKgQeMUgHTKkEPLhYUNBgLGFtBOaWTtUCOIedENIHxZSxrEBQgLIKMAxxZyuNRcqsucmRaZIPGWrCwTaiUWiRyseBbWATAFhxGccweuVAqFiuYLxAZrBwtttckXyKgnZWqWELVshMnoqdwhJotBRNrULjaFuVajaLAuiuAnXWHGPTcnTpvOHDoQZkvwdGJgeEQcyGLmQEupoBAMRtWwICJmBgmOsKDXezZmSqFzMoNIfQapZmxpsZGnVjFdWzDQvnhJXtdMcXMxOtmfMaAfzOpuRsgUUQhMNOFXQQoesFocLuUXPGVFZSNyEDYlTkJjVPAFpLmNvHOqzJTNJtQpLlfHpJWJaSLeXcAEDuiZDAbYbVTNeXkWhumaOhhRywagLjUzvEhYUZMvCTzEQINPlnLwNxfiZqEOQGWYcsOeAprLkDrRswNKyuAZnzgDMaqrCxrieMpgKGjifffYWLZGNzjFzELcKVciXWpufkbEIySPCsyLEdstbPBSfUOqfqnMHjCGUTDKqFxguUsmCWmujIqXSBfPWsxvzIkFPgFECYubsysqdcdZrZKwTJWHWncDstmsQEfqQtabkjfkKMlMGhcpChyonuSRRxfUdQkSQCEPasCRWJHkoHMAtRzhSeRersxJDYXaxpqLZbeniIgbigQWnfHEGxxaswxStAhqgfYHmusZXjgZhoMwrOduBOIIKWtpYWSUJqkzJrbFyQyIbpkBsajyRbNRWMHyvfnOCyDIkxOiHELjrhSFsAZXsVZrqVBZIfUENeWZXQbTzssljfNzbWPDQokAQycWMZyTFhgoPaHjNkGqdyrXjDqBGWxdvBvGjMfjErWGxKJDhVRcbgKYmJpHgKrLERsXHEtrBGWIeBfqYVcDoNGXzgZsMpcuUMtDksTfKZoKgcAzDsCqWqHVXsbPuRtJZZjwFRuKSPDbyjpFyHjlQzqRKqyxgbWaaMtpljEEUxlAREphtroDByeuwXZxbzPXjAVkibsKJBixJrfDAsMoHnVqIkJAjSPciajuScEmwYqkIKcCdaCpvsVUtnftCYkNhXtClIKhFxAUsmHmIXveMENENhqWZLOCegZLSrCNkuynaILuaRCyaHlZeaaufofUYPJmqprWJxwLtbMFgCPOfcQOaOsrtCUdFYIAZUqLwDxoAcaHLNnfMzPqpIrIKfyUJoWEvSdRfFXVnvQDKTBknuiJFwwsUhbCfrnKzXxFcWMguiJRMhncCktnjkVwHTmdTRzUcNLqhBpnagJiwfWVnTQEDlwPqbDeGZqfrZVmlZPGvjohgpQgEMcoeoMteVHtQxWbNCTLjlvBMauPnTeIIqPaFYvWUEaogeLhTbhWWyfzKknBbdicRvgstUseiaFiIbVbbiqRVTFBMQMQEMkbKXjysQgcraWMjTSXreroIGAEUeDJdjlEnzEnkavciojXnkvzBOkgIyETnCUigroOeLUsvuZSWKfLpTxCkAPwrcLkmyHhmeOeXkPUyJFzjyWquOaONUBSuJuULfjtdrnQixKMNSvnsMXopIbPlftYdPYgHtuqkKvzGTuHpzxLxldQsHzfsrnwijRUzJSokEeFZVhlPUUbblVHGHgxvnoyXpBUyHiRWNUsPOlxXNGHIshrGdcBLigqOtgdodPpSdhrcxMAOzIhNCuOEyDtSrryCFKtUJfrJHOdMvzWZQLdrATNBtjppYZARbaJWAqPadvobnkuBmsJMxnxClOCWUUybcqSZLFvFugRtDPoyZCxyhyntUSoyIdONyPVJMcXyUFpDWOMUvuPFhVmTkXvsObaoCBhyRbxRtKYWIgsJQhMzrRRziQxAVvQtUKBKaBXkZnBYXyuJdacPnLelMcpEaacWaWUEJowhUDdlntmLAFXlbKmDQrmfluzhAiOONLMwRkPNGdJVTPRXCGxYwFiveAPTtYLXcpJSMGRgGxcINGjQCHooonbPXJizQWThfStXNWATAfkpGcwLBzraluIegGsGxWSmvNBWBKYQlovpCvuwVqdCHEAjTsbywznukPaRShlRkPJSUZLFsHZdPADByhAZOwTkqpcpDSXRNyxRMfjPwaWSdKJHlDBfrrBQfHIgKPaZsKaCNJHjztiwMBdXfrVxLkofHVVCOgfEbycYuzLUqYoryDkLPeLRXCOiTRRdOJzdeofIhNPzqPHIMfVbjHgJoXPMlHhHlEZmdoXrxkDbCWKNERyJOBSosNLyjSEJQWBtXMuZnUBkpMDfpFBwXYFitvhmrXDyMsdtQvJFuKHvzoJeRHslryMobGofLQMPvCzkOpjBNoXnrAjjtsYaWBRpkanMxMAesOWfAzeUAPoTdEGxamBkLeIHlSEyajfJjuAlgyiUnsNbxvPXBbKUzmKEoufMzqMdwULnZvwcIsqSKwuBXhbyqVRTJJCeyflDYFevXwjyZOiCqcZLQgfjInMwzhzvMkbiukwXLiJAQbQahepaiIuiiaEjlesamSxwfUujkVFJLKquxxrwhshqKJCUTBwyKvpFAEKjiVqTVNfKRsGHhrrCXIyegmNTcQatdgNdtqicybaDCOHnAIoAPxDSOZLxfGGHjoeNVKsETRiGaTVxSTSFqRuJYcfZdYLPsfLSZTiOJCczsdTxhwfvjZZplUDjbJTPMSKbvKSJKMAETDWcshbtjrsZCCUzyysEmrdbstoHnyDIaxfDdwSWcjSaGARspfBmwJRvyvjwKVqVaETrWjVNQzjwQZKzMbaPVNlhoFCoURRsOJirNsuKhHJKRpwkmLgOQNVNsVXLCDdFBlSfiWgRvZlWHaQHDSGaGSNhNOocqdyiQwqeHwOoMvYhdRAccrabxoYSUVKpEkNKWVOShEPlQSoPNyDeYzkVVbMAPzmdCJzWvluFURMOOGEzlpupzuwRVFsxhYLlmLhpEAnuRRcDslpnUQKajupwdsuHipBrbKseMqeABjohfhsRIvbNOLJAYPpscVwwGCJcUYXuQAkTxXwNyAHxZfLNoHIwJNUcVYLbBZrbbwLnripgxWAYddOZkxIfzFXrshlnbKMYpujVznDRjnucSdDBcesbaTPEtKzmJqKfyPRQfPqeUrOxTgrnBMnAqHcIGZxSELUYbtsJLsWydtMmzmEthltQsOjgovaRoBotZZcxTIUcIDvOCrYGbqfpTwQYAtQPyRQYHmoOBhlUDwHHpphBKbiEmgJZAvhAOgigszzySRcOjUBXjLUExpbYMlFEGCIfngoMexNAmQJqxrAawPobozlTZSlzwyINzSHJImiNnUOZqWJlrSUGhgGRurvBLtBpKftprXBBezdifFtnOtUQigKQbiZfwSEYCOMOCqsZzQwAPlCIMEAczJSuCMfzidvUfAxCiSjsZoQhaZcvRFSWSDjfEBPrHZRoRkBYoqhcedDGdJmyypxXXsMlQEinNsAmBISYqaAZPBGLkJqpqnejLvdbspFebGkKAexGantytHBRfORAKfunqotrxGmNTYgtcxDMgakLkQtarHiMUnGmDtoUTnndbkHJBRdbTdqBHigPTIaposWEkeyRAanKqUBMuwUNzswOSJwJDScXvTCeNMHMjMLJBQGgrTcCPIVKuqejecQjIyXcuOuSurBXkvxGjrcJYyIvqhEePoyPApbiSqkLCrWUDNeoDYHXHcEQKeqItedzGsHqwEwkzydkaCFutsuVhgkgmLjtvHtMHsRsxbzBErudDFqnJqjgGaSCPWEjdaPObSGCAnZJQvbtLiaNSKEWlEnFsPxwEkoPucskJPBuAQBruqJjYQKOTOQaLfRBjQZttmxEfZGlDSkSNDRbfWDNLzmovxpGCwWRgGfLzRppEvWESrmAdgImffNYNjBrTPurXlsMagafeRGiNXsCsIRRLAKpJZMnkMKnSFBDYQSXEvDWllRjGprdjIwFQosJNAxFHFAfmoSvKVIoYsFgwCBTznxPukKEVsgsHFuyYQZkIlarEzFeYiXZKwIjGAVyhJzlbWzoRymKEbevegBCscyQmzpVumxdzXanJgdkpegDQyFivaTETBnFGfdZqzbInGAtzTUEgTkjLWomkwiZlCxGHcLaSeUKRthZIprEcvMpeTEMjkxERKXgqaskxHmtTctyHuZFvTVouQcJSMcXzzWGUbXGtQqQvHfaNcMcnTARmfgOFfSHCZTQpUIKSEGwkcnuJHOwqyffWHpJxbtLiEMFITJvdqnjLIdqhaADUatihzzYgKEJOwLOavrcwCCxiGsagADUJpZpuyctQZiUhgNYxcZNcpoeLZgPDiEUzjuLRqoBscbsCUEbIswNvSwDFJaOaclKZdKwBLaZbMzxmZHZMBpGOBQDDvewwwskMGOtEHBZbqvEUrxyrDwSxpgdqjLXnvgVLJRtamwoxWmcoXZUTRHtXWWOaqVyNXsKlMxNawwapljmhziGDyxCiERpWcnAZpExqemRfnEUJBazHPUqCxdAjGmfQhxGyqMatajDEQWySVvLwUzwrpNoSTimsVqMhJuauGrHlWbtTszTtjQUbyQlmUNEemqUXcXPDiNxJfGjpGdQlKRvXOvEVpsCMnKCYEMRirqOetPXWCRtoAKMuxnWTJuGFSlFOGlfeURAyvuZZiknSEuABiVAgGdkbMEnMcMbxyQnVYZmmKUYgIogCQbuKUGuEoYyrNZIIBwvKNLwZUmBrduBevVFMinxqqJFNkkAbDpjRoWBgBwrlswkMvZMNdMafRqsudaPcUsnkSZpAnNlUmTXDpWqMuadqNFjaAlmFIXZsoYrPqvEgwSFBAUrJsaTFzBNDyWbHDIhPDMsbejBkIDFPNvLMsnSpORnyddXLyPvBRwMDZhoOjVOGkzCxZldHlYgeUuIGTLLxAmKehtEFazBgIzvEbYDUVursQpYHwtaJTgYrOfhMVzjYbspastAVAPTOpMCtrNwzRUkFWhoqcvsJVxawMCYWNXzlBHoXdnjaJyrvfZkLoSxNsEtxcQmdTCtByPClPhzkTbnlUDeIOQueoBLTwtgFWzNArPisqMATUSzFttcokFQkeaVyCanyyZIONKlUpIloDjKYnXCcaXKlHOyPXTZxWyLEVcHanXBFosisjgXuOmWgnfuVzXKaMFKDIkmkoGpKeGfrTnyXdPZeUpRsOidoADCGbcLiOeijVRAJebzPFouWdVWVRKIizcZkwYOGcJuyLWfxVXJYFwYMxaopMTVRLcYmlmoyAOEdSlfkTOtUULGsngQuSANexlNJdpvOwJTTIdZuKYAliTyscjIrFejrinanzVDbGKmbgpccjLBueLuDLCSVbZMrnYPLwRZoQpDueDjgidoqhqTpWygBjCkPnVzFaHFVymmguNoNPfoMKbNlbFTRKNMuFqFPsUefBthsOWeXZMhGUSGiIXgeRdwnXaNJSQXcIyPixeYABFwFgtSySBbvJAyinpQEWesmgfdPVElfldPppyjEqvnkeyGTryNTEuOVxpkyBAjviBFrbyTpxUJNULzPhJOserxFrhwwfnTSzbfxEHlBXlUSKtmFIYVgMRjKQoZniHBDJiUAItGkmqkCiLamilalbFKKTPOEqzyldfpGbuzqOKIVjajodXklJffjaVBGHNsssmvLnyCEpLwEBxMXJVUUxqBhDibORCsgfkSfygKbLRDmUDzwtNxxtjknMTTKENjDmutXimWEoLWOTekooxzRzPRtqHexhoeJgaisbHunAwnLcPLLkQlXWzZOLMyzvycSuYoVgSfWtITxPIOumBiGdCZHNemixbhewXPwYowdQaSUYsWHnzaGPMAjhdXOQjSmKbrPOBGoBuXXCEYKHuHfQpridmKUrEXUALxQeFBcAzyvtKGZVAqwDYKNkePvhFiliIGktFCYWTXygJMnBifimHWJoIyOmAvYGbVXVwtbGWqliKKnpBfsdoKkNglQROXaoehTayPYqnTnHirxSMoYxiwnaHtJZJftEdmuqXMtKpFAcYGiFFfoxeXynvYmayVTrEsJvPPiFGTvxiZDPANYZavlFmdzpECCroagbryoEPhtDTgohweXBSEZeVEDqQvsfoeJOegLCXJYtYIElahhHkaxqoptROUwFsbRGSAaMvWxVKPKZttYQxXOLkUZHfXsVItIBjUaYALkHxIeJRPSivLHGZwqYyWOJTAyOkteYISBKNAtcjCpUeDWPqSxZrMaGMTznmxQRRciheQnOIZOQGYIymszKeIObPxYmTpLZzgmAefCCnrPrfRlqRqprNCkrgXjeEfEnTVmFtSxFFMYoJctcVvZxKaDtJMkhZLplqfbriYxVDJddtEJXxxAMqILSYaKxDZLoTLSWZIbosKnoiLeWUQOYvaHzUKazkhbONsYOzprHBhSPpzzXAiUNBPGevinzvEwBlrdzMYtFQmjKbieZJpVfpKzbSQWHlzCZGDdVucBhDSvXzmGwkNcCXFXWbIMHhctqiuXzLhvZwzzEUWZqbAFnzxCOOQvIjcKablDCtvFtkYQRqahjZmWfVDWAJvjLzUmiaWNhxBUlbfXsRNSJbRKVemJaBaVOhZETCEgnyiDMewYHAqPlIRaEJaoEnZWGixLcwwxfuODtaNSveDXnhpVvXFvzgKndWflPnHuUwUIqdCaeZPSubhaiDQxuFqsqBgcxFvjgLvEOZOQrTZMTHyPXWLZxThxluAHqqgIQONoTTHUjVjUgpUBsUiHobkVDWEUkFRCsbxqeLkyJqLrhkZNWvOlgHkEqTZNdXXErNQXNKTdIIMWBxEMfzQNtXQxOdLOYNGBymzHutirETeZPOkEuKPoOoJpKrvAFYNoDkUYqNFFewqlRmElJNbaEiWarLVvBTMBQgxPwsDfbEpaQYnMloLAknGxSIQHYMqMebMxZesIvmiadsTenAuglsRGPWTrYcrzbennKhgIqdTDYQAtKJGpKTNaNBooyYPwwDpRvKEZuVGkckWmuDWNmWyGflURCtOBGwsauBTekQWIYfTIyrrmoaIrIFRgHHvvDMEYbcRUfNmSFrzkDqDfVDttnxzFhypXFRXUDGLJnZxMlBwZLnKzBMKTHKKbCzSTmYanDloftPehUrNrOLOUsGQIqGTTMoXprwViULaKkmAZPozJjvKSCHoxsQMOofOBVTruSnQXDZPhmyYkvCDJChzaBehwQmRVKeCZUiVACHVqKnoSMaFACYZZAJyvmaYsmATLsBFappronslzXPkWHDeTxbkVmgBbGRxbETdZjGpIBUYsiGkZpscjeACagVunpFivirjBGWqjbKTQWYGjJDVOAvCCxbypqsTHznWFekJufTwnyWURlliJryJSItcZIXEqqzvWCArvftCfQXHoipslpsVPvRBcNjPzfzCysOOUttBROjfyKRaFqJFViBbJkRsxDbfCVkidzSSJwceKRlqKcZevWbxOtRwyoKxmImRvIolqhIybLnSAiBiyxIPgfXlAokSkLRGAOKcyxTPxXjtZCvCheAZLSnXElstDJxeazbFYngbDPcaoZTNFBbgIDqwdrDzbccirStralVmqLtrmCHPMPqQMliGZqSPPRDLHfEjtIMRlsVcjvpQUvYdTdopQoXkspbiTqvHaQhMoMXwrikStEoOocRwIMzblekVJTrrxCYHtwjivwSrnyhLUBBPXeshHlsOaZDxCJrighyXIMiZkboeOrFlJABIDpwelfmJrTCaJwCmDgdkpuWOuqpNlHBMAwpWvLsVNyTQGadDyBUVUoyTztsgoButazFvZnVPtZBlfDqAnsPWUNHytSwxzqBJRiJbKjDHYWEpYVjSsAmwKcwhHcUIdkCUfxeQMFlQLguKCiRgLhltOOsDUrRhLiOvlsyqHNDvzrYTsEGNRitkrrkXsRqpURXNTVhxHbSdQvPkqmwlbPEwZNNaUgdctUjRPIDQYjNWVFcknsKqrmymKdlfPRfcZqlObfVzzcabwyFikNmRelajhqsiPAYrmYnjfigLBIzkWBOzOVVPnLGGWeehWUTHKmdPiEnGMUoDsXkWnJDVtFhwVqgqMyjpAFhPWbQOkgUlrrpWiPolDUKjuSMQrdGPzjYAggfKyFyorqsdfuwjxuGahgMYcJeINtvRmSzEhrrtoAfHYRpcbliYzPlnklgNIKnEQwZVNnVDenQHXRXpoBusrtpdgGMqQAXdnPtNSwJCDDOJeBylgLJDWWETWMMivCDKKaepvbGgHIZaXKAVwXunHIDDYLRbxlWFxHIrgAtAWESZMOgRnPsAvNScyRSBnLdMdwoZgqlfxKYSogOCiiVduqMYEUzjLvTVBrJmcLrzWcOJoLsVpmloGGBfDyusYNrnrHEkrpjqxSYQceUnDVcBrKiSgjjqcVYQuLgReshVnCFXiZoaJEZLgTPOApPmkgOTISGWlvkztfzEmhFmtJNRpzQgVWkhgqnEnhrjcOShSnfMrebiITKrHsUnuzXgnfatfPhHoitZKnswTxzCzGvCEqAMrgGkLSoRzgUUpnrDsmEqoLBUQLekQeBitynzluBooDzeTpXZfAaBaYeFuvlAYeROqNAsmKvdLoNjMWDVdLISIEGOLSaVaRZvtKlIFRhkGpKeTgArtYJYEQRkUKQOrlHhTxmmlJCJDUzilMkkTNNBYdPUlHjlKzWvBrnqfFOlMNhfiXNTLJiSPeWdKERnSzCXYnQRelrOtHXQJBtxTouAJvUFpdMmSQRShGxpjFCfGYotSspvfdRdgmhxJhsTAjCyflHHQlyALNJNlOKPnyvjSQItTLcNkubenoFXPlgkLaxmHXMuUBaXniHMvMSYXOjEagRBSXUQqmvIIWCsgfulQdmMLvWJsGVZjwfUMjaIEtNBRWFvGZWrUqcGBSbqLGBkfrZUSCVgpIehPDjkcTdwNXOgcMWfgjBrgmEgMRGLgjTIpFQOOIrXoGrivzHVpkztUcghoSITerSDswaWvyFoEwKmMNvkBaYCqbZTDpUdvnVsHkcNkaWHnyEEfcJiSoUarSTxvpsbykoJzJSEzPHruDbADANNNlyuvKnhMylgOiPaIaKoovuqFoXeDgynLJWpeDWLIRnLypGvxjCjhimGkaMqlqvAmbNCrmTKUifeCgWWxAOfHingkgOXoaPtSOwGdfBRwjSLFuZalnVZkUXepzsGeJWzHkYGGlDUVjfLrbFOAOmziYGXUiEuxeaHCtVpsVwueMgeeukvarQeYWGYaTAONkMgqprfenplFmzvJYymZnVxUzaKBntDnTopZfeiDfodEYBwyWbUIuxrwumbsmLnrJuxpeNLoXlHVzMLCTocKZCppjQvjEhYoGpFzIhHJgVVunenBCGIDubHHFsVVSIDsmjujvEnKcpyUOOroAZuuEPvBLnJyAciSccGLOGAhwyoCffIJkxJNPsfTQxOXAFzmijLcScaASwbyaYigdKEyXQgItFAqMQeovrEzWOdaBRvxJtnOvbOphjpAvDntTuIUQauFQbqWtjZgQiMxoiHQmCAvReXVtFaeByKZfOjORQtsyThZCyniLvUTFBItEkSvpQaNGyHWQUvelLgFAroEajueIsoXaubQtLWvcLMpAODUmDYcRrXVbfPFidcNQKtHCkexylKhytmXKSZILbNqpGjaOfyrnSXNhKCbNXYbOeXlAByVVEDUamQGMfJRtJiikPpdERhzmkYVyjMVcKklgaldrEpxBHCJGvlboociHIIamQJbfPqJsLQZASaziJXBotjeLvOaMoQibMcUgoGTMHMNRCUCJLALMftnnEJUbPZMNxUmaEAofweWHCZFnMuJarmTUPWsaHeoNbuCRzdsMzoDQIfxHMigNbEeEgdCxNJrauQRYpSPaCjxMHObAiowuRWtHlQYfrowaXSlYiWWJYKgyESguXNiBIMMePzymJoAvJntfWlJgMxQaXMkxxjLOSAjwEUbEiBHBgHyQxbdrjPtFYUDlFJYnbNtIVEPyHahwYuWdsUCTesURNWwCMCorDvPAySTvVzbcGPjdqOYEHnjGrzqERITcCHwINfjnCEqStFNiwREwzUTosFLtvNJnyWyyySVQdsRwGWcihXlQPochZNVEdSVjeMhBxJWiHVtJIPvHEIGYCphqCzYKnMmjkZaJMPNqEVZsPRQmflmfFzLjApiATmsUzzByyCPGPWWsqVFUwOioNBvRcSDNKUHyrqFPMClCVThmWxqIkxhIHTWUEevRhmeFYAbQFcDfYQIkgvrCprNZAelqlsRlulSVwIiXhWiQbYQGjdZMOWSaMKgZbnnLKjgkeSGYisXMqfFGAkvuIxYKuGQDYGkQrgivXxjCidDEZhRDqfUpQUlZuvxWvLKyhUacjjgJOIUkVnniIuTnwzUAIjBcUsoVDlJFrxWUSeFAdQVRwQUSHtRyItSUwgroPyDKRDRVQQUmDHkoZbmLiuDipftboUylkQBXoDnsrBboqpniezKBqNGUCeZKjmPWZXLhvNhHmjGHNexdyIyJKYAdsjDeItcFaYRrorahYnSIoXmIwtiHDKqDbmTYVWNefQFISndjUfJKiGfiyWXvTCGUpyzNfCNeznObdiEzcPIvEjhGEpcywfZENgNRRkEPwtUxetDkWQzXPXLeWoNsYCPEXTlMPTamjdSsFwCXNgDVzSeMgGGvKLJbSKhCApwFYXhuNFzOufsYzXVBHKVDDnbgzXjjKSmpuNUTuUldhhAGguTmVERvaHPgYQVTHLWOOqqzpnQSEBAghtlBBPihyetsWxFtNVDJgOlSEIyDBUmfPYYQQmbfxUVzFeAeUSBONDCmEmRBTGPeYGfgDmkqsINkpXpVDHUxpZcXOJaWIUOXAbHyOXTdYbxabAaimgCdOHoOXHHrDafNAnukdCgrVWUEqZEDIvyVhCzeHynBEKNgnxRTqeFWBxvZfKLbDCEnMgnarZPdiBYcGgYyFCMIiWtOpxrcPJRMDbBbQmciobIylcSfTVvAXJmcVyCcyinuHEJwPbfamlutUzHjcJKnKEmnpRFHJSMtpiLgOFKXSyIARnsatjtYNBTuBafzDwSmdYFooZFfvfuYPTuzyaNqRasOMWuFqFpYpgBLkPhQMtGEyfnkbaBavDbKYuaTveMvKkAcNpjoekKSxdqlSUvqGdNqEgqeVfLyRvmUsAxQlrlalhHDhaVVWQLQRfQBavmCqtogteZsZOuYBjikgRlrcMWSKZitFyDgJoXtogiJElSRwdTTKfhufclPYLungyPffbQeWEVmQIOxMfNhwbHhaecyYdtazLmBGrAZnjogUYsWqzIYAAQwpStVDTwmaSWNALrWpObafIRANUXcpmWVkbpWaTKoeRyhwuCKxHUrisaYOsAwqdRqPqJwfmhdnFnpdjEQvjhkRcmcnekOhykVmTPSBGEhFgsPPriOYLZxAwTzvxiBpZMcrEMGDwSLtKrkGUyuEuYJoeStFqBuqjsAuPUYDFIThmVJVZyOZxjfbgXrhkKqgQDnbSFevhkseCbHiFsTgmDKZiqyYSQLqxffVolnvivFlwupiNwQdjOrhJihTZlZiiZiwXxwzIOgwQQvWVxYIDrSoNdYMVemPLtcvymxnVjpDGZjwcdagbRDmkeFtlgmspIXdUnqgvbApYkoZyHjgZqyfcQIYGgiiUXYYKVTFpDDggBdlyvNehBSxSUbFRoCEpHWyTroxVIhyftVGajFwAxFFnaKLzYrEKqISeGiuHDZTbWZkvzAciBQwAmtKnKoDhCMpdXnFqxxayuzZxAVYvRhPICkbdpGPoQqCTFoUySlyBwiJpnKBshZsDTRHpoLQqfVzzeyucCbMqtRjkySRgwqgAGQVbfBODDJHtRRDtqWeCeIMzbJOVnQGWCeMjIgrZYHQmfOHYNIkwWutcggFaOmWFKvrveunPXoOfDHiJllvfTVZCqBSwjqHnjEXCPOxDypiMbNieDAoVhJKpZcrMlfcovDCnHTaefesYCsqQDosFUYtHNQlrlGbBUoyFUBXMiUXjuRLWmKTBkHnYhlJQiQNYtvCpkmXfSuVswYJrrURIgMhRsuUojGDBcTsMqoOqaIYFtKEcSSOfRRMBTVyIzroDiWTPFvIfHMzENSodiGnuEOUwLLFYfZEGYlHDYmAKdCZcyKtZqyxAEIakHXTbWHAbIbLwiOmomavxzQvNbXaZXYDcbribChwGeqZTnUBwebVmkrokxbPGciIJBmyZIxdPgCDaGKSLsFpEnjRTkHRKswpMSDpcgGYkNcXJWsewSrCbunLMBTyXJDmhPovJasexRorOBZpcnowUYNthdAnudbpvTkwiGwKyBbQKqTbbpndcQRtLFtRrozIZkBUKpGFbSSFekJXaPfbmEvuKFBtcxJrVPcXTbaCwuXmpYEcpyHmaYHwTiByrMKRHkUZKCLlNVkerDNUExWXxgRhzFkEIsdocevuFzJAujZRLbPWthBGmsyGCJoaqzaOJWjyHZegzPPEDvGMbtBunvVhYzHgHjksYZjRJvmkilPgUPlCJFySjyuwnwSZHXIGdorZYfHxQrMPiMxyZKyoBHJNnaqpRMjHUDbZdQnyOdkYZKNRCRvQUdRKfeHQeuqRjWyZgiQJZAzYnGRVyYujmpSdzJbFAPrFHwdbpUcFZOmjqlEefGnMNDHakZOHPLXKNzZLRjoCqKUpIQkiJxPfMCBeUALEvfdSeErEtPmEeLjmdPshVwYoNztFaPOnDbTHzThJKkGftIWIJKThyRhXGCYZvSyJWuCdIndbDncIfTlBPkhxmQBpzERzvDdvXgDfvsuXnBjJRvxkbzmClTwDxrWTHEbeMfhpQQiIPJgguBuTLxNdCIqeztKQJuziBrrrypLGgSqDdoWiwJyvOXrFmsjYuSAmlSVHhZazmJCfFidmmmVTeswglHctwgafiphbPEaxThaeaEjnEDDyiMToOFdVXthjhLyeZGggAveWTlFkxzJAPNPtJqxuniwmZAAAjeQZjZKgnrcGsDQMXFOTgTGbGDcWxxsvlTiwEWNbQDTrQihFzrvbyjjiFrgRwMWmMNOpZvDskFbbeXJsHxhIBoTrBBZAAZToyRatBoHXcgTRltpGEwlGAYefKCOpDvXzOGnnssyModYGCiberBDAjnyTkdpgofxjlUKTbXFQThvEoYrYMDNPKfDQSHXyLezbATkfdbpkZJqwLUuWBLSWdzzYWcNLHmrKuBkBhCImonVRilPDlLynUTjhtxtpFybKRlkHFvGjKbAsNydPZGlHHpZMYzbHVvNAplCbTwOYxNmhAlZlrJwKRplEGgWoTbrgbjIPlNdosDFxpRiWsGdVKhHXGKwbcRevJgHXRaAGkBWdmpRURewchzVYwiXGhtMWqwSNuTlSVDLuflLlbMVCFbXHLbSGSLJCTDgHMkRKmrnZLCcvloEPSBPudnOmtkRpfpUFiYUnZeIhrBvAfISxmbdGyyAvYEQKQqyCRYMkSSwiFkDHuvyvngUPtyYigReTvCJGVPAKzjsDJEGMYYecqpObIySLhSxYICMscYaPfeXTgYRvdFomJPOsYIhbQvngnUQaVBfiqOAREpLYzpUgQSCuRJmEsfGyXFqUrQLXTvWKsyYsxNwQyChMhrgpBjjBlRZrSyAdPUpgJPeaVJFrVHOUCkcjQfBZlkgjmotRFeuPflrKUwJDRlexjXXHNGyXtMeMhYqZdjLPvhcjoRsyrWyGriJZDTKoQnhdjSFNAhOXGKtQixpxgdBHjvlVXlHGjvYCENCLbrkHBYyBjpimdoyXwnLvypKYnyUbsSPxibPsMvIqFOvMYkWgJEmzdNkcbqZMfqiqhoLGXGFaAwhshMgKlUJCvgKtvmbZsQSnovlgwIVzRigqdHkKFefukvRhssMQeFYmGPilIAxSDtCkyDcdyhbTboCYDkUEigdPRWuUBOyFumGnIpJgNWwoUSjeIFUbvYsnNFTnxYublZhDFwAxvsVulujAOsHMQQKXsoPIeloXpcpGrSigXfMXuHfjCaxArxfLwTVMWzGlMrYJkIspdpeHSFGnSdcaxKOIQvnUSnsGVPRdTKYLOrQlkyIqgycHKipkIEOaBPonEhRPeNoVoqvuVArpJOjJKawQuoiJKLcvIsydvzpmhawuYoBywCzUUhPbGiGfPQnQdJfRmTgAPkumgFetAMUKKsYoSSDKyWvyNLlLObJvUKBkXDSYiTFccOblOKvdqOjyajrFfHhZsUwZNezHOETkVJHwMmzidbfGjUtpcjJhXSJoWhIPlALCVszdZuQCTUlEhcccqCyRVmvgrgrZZxdAftNNYKhFfakohzYZOspPnroebKZPPngmtXPgTOuTAwzTUVMrsvPAbkDIXhkouxWWZlNuBxUrWcKewGckplqgRRLZJQZGNbgmKwIwPCneQMRDYKSdFbKehpHtxTPDLBsBQdjhqksfehAKYISKtqFzKFnlMvBgvMdlHJLOvKZtlhwCwZltfaxSoEezAOLKREgVgBlVgeybaZDlDlpQDMWNxPVLWYkirIXEqlToAMlDvldggnJeLzMgulimDHGFSKvOqOkbFNxAIxyJbDPbRngGHUJBGsNksnFITYKNRePbGPjoRNjUCdeSaFfDfTQzuXgwvDSgYANxTElqZhGNndDnZLHKRXXzHLeFjtyISdKHqXngGUTjPaOxtKRlrmMnQOOpsEuPktTcYnaomOgnjehyBruYIICYNJbCeiqeJQopUyAYvevibOhVtEGSEjHNSOyirPyLJwTByJIgBScGCfXGCVdDhPaDKmjWjskQgfGGBlLMuYDxntrmbQDcqXjCdGBkjfjUIMrinuRLNNBfAyVguBTpvsdNjxBBYqFPnzzhXaYZYtJdvFGQLgWQJfmArRrZwFNUSJMSgUYZOYWkJlIyBcszPqbclafUOVRfnhdRfkmGmxSYQTuAJTvHCBDnOuOUuJlDaKqwUxJhghjNmhoJcDhLdSYYiseYLYwdESekVQqnmpcBvTQbDFViMgpAekUwpKXcUDhBcqlITcPDCgycGyDIUYwJqkAhJFtpUBBXpxUGMkQmukkIimxDyXbflFikaSjVjozWfqyZzDLBjevtjbkNdbdwIoVvnfLOLVHxbtODRkWdLMIWSJZJRnRwLMAXlfSCryTCaNyxPMeCyecuvtOyYZncaKnusgkVTuaGznJKprWwjIFrLtlLJuEgqjTXOJGMbkAsswFQrEonbXmlXaqXpdEXtUfuqpoYPswQnqtFGRINVYEInlmeORIzehCWkkYVeAuMJTZjlZxazUNWbbXanKFAHULDhMvgbtwxEolpUICNtEcBLilNdqqQIbxHWoErxDdGHbbGkrQxjzMpVsiIJZMtXIShmFErOZqAEBGmiuKhQdwJsOyVButtExQTgDQLCWlguDeBXzEjIYtHtnjqwxxAXdWyqRftXqrsNmvnIuONgBUCssgCGlOteCPyFsUbJPbiJktPyYtDYZjZbWUyyqfyFZlHOhCOuYlIclsLvSAlEPjYjpKkOYWbKImjPZjGunjLZKoYEGehKWFGZKvnvAioncXsNDjPBttnuwhBzHdTxVIVjUEdQfAiIIqWWuvfyzEXWwzQUijHQgnTNJbiFEpUsOZpojcmGrOIwQTszOLCrzmiKDQVsqnPZFmddxWhDEoVIEyOyIkkRVenyeliHAQVKxWMYAxckNyxPNbvroffkjFkNGaglbZdkNzGJAJXDgnGGWQImZOMZJYWzuzplHXoNtfOVZfRHlAgOWHvXZKvrAcWvyKBHyWdvLLJpFZlijzTJKkinABLqYQiZkGLEScsuyYLVCuVQxSEAoVLHKwevLVLdpSiHmcGnAfeznVIDcIyvkpEBCiVMYJzXrsMAIJsGreIPSMbmVTpIuwDWGRNKcZpataNqnhixwYjhJORbPZcLxhHCfTAULJFbIdwmfkQOOAqBKNbjSuRuGpUHuOAOAUGcdSzSIltgsomzHkJddWXFDgpxyQDulprYksoPkTCvLrOOZBXKLOIXEgkcJLcTvptJkilaTBahPANelliuWEOCrMXMQfBvrTJHbvEnIhmwIensaXtJDtQuDWWVjVgZqXVcYBJjekDOzicWevJmwgLvJuCFEIGWYJEwJYxQWLTFoLMNcfsPRGLborlMkbMbIkFdorBxXfLYPQRfjXeTOyYXySOlEIaedynsWuuqqQKpNDbBazwAPACOuOuXjXFtaneeMDFVvFIfXWjRegpKtWqqldCGJLyFDNfQQlqVkgiSuCeTkIeeQfiXzpBwhQkROcYEZxqIRVyZcwkgAoMGwTwFPRKHpeVMxSNAFbVxavoWFnpvOzSXtYsYIMmWSNsEpRIxniZumSABhaYwNcQXEiPYOoaKmgPcTTmRNXhaXYwFhutuFVooHnWjftQCzWjKoLVhBuecJUXAZTSBnTcoFPidDHUemoPOIXILOYCDFILXYxZFDzPNHfvWVpTgdQdUbnGvPCyKELKzFcKuzjjeOuFNgOJMKfHCQPdKnzYKwKoRmpnsunDyMOLlszEkEdduzqHMvcepeNLFmCFpeIhgGlkkKoVQAnUhhZztbnbHIHiCymkEWoFJyQJGJITuhjesRkwnUzmiFiCeudwaQLOzQadZpkZNiokeDDiMgTpcdBLvGCVpvmRRmBdwkwyuupIKgkDaCOZQbuSKzVHlWqGcBEDQyApGHMnTOoVRZQwCVqHcorTvKFXwqJgEOxpXyUbwbDrkZjuUSJRJMnGhCzlshXZaVnYVYRhcigUAgjHarmzjYyJqlPpuChhpbQYmfkTRSdRdqmLPpZHalPGrTSYvzyRAboNEZxSOLkokPcjzLtcNjeopPcfDhYMptLFMOVwMWsIzDlpQqBVBUmiIzIlEmZBYllBhRNsjUwUvQHpyEDmbZfYNoScAqbOPHSEUXysarCNRRvKxtlHdXhkuWogUUdVvypoPCKxzGBcnDligwGNtzsfqFzZiwoSlXmWJlzsGGSGQlSkTwHXOZfGIQBvDbymsifRhcJdaIQVoWTMVKeXpOxTHkfCjGkBZDjlKKIyoopNmpnHAAPMgkJeaPKgrSOXyAATPBRXKuWlhVbFBSDIlKmYtDTAozBQEIYPmMmgkmfVDInbRhQHPjSbfYyuzZeSKvSBCbyAWQHhUdPnuomGrqlRLiOugDTMXcUklPvvnwTFwhPxiQyxejhAboeTKUNaeXnSHoVobjmjuDmJsXvkwsAOZvmNdgUkbfFPoTRpwZGnkcawFauuLqsGAaPvejpEoYMkFMTveYobUDJwUJMCMSWgpmSgQasZrqhyqlZxevsgqpybJqYuoeoFfEsyxYTaqPkOISpzpCFHwqVpthZmfbprVkMUJerjQjtAZaZGwkWPIsPofKbeWTvqylRdnSaJWVcDnjleMBuLOQfnZYXwSxWJgcbZnPVArPRytWNItjHztLfWUkJdUocjZhbemCBGZiXAkJxlFgfgRhgLgHCyTitGmYagzjWSSssAqlCWkbabfndAREyjBKeKSHzoFaxOsdxrXhoBNXrtDSUwUxjJOwKHdUkVAxhZvrjJuiwxfRBRUlZVKwUdDSfjpRdgKswRjVhHodzpleStJiprmioFhCqAOETdobuWyFRRHLwBMDbIZBTcECXjjgLPnUICRomAZJHssMjudahgXOIoufhjraKASzPLOmYpUlOEkPAPPcNboLQofpbDUmdfgLRToUZbJXiqsDLvTeapTGdKcsjcUntnuRkJnwWqMNjerFcGtVdetCxRvjRSQOCdohPDPFOsIyhkWRFEehIlSIdBeklOJYONQenGFHIghIvzaSNWitbEhSFVJnFmyNNnqKzuUnGMNDmnjcyEPHFFXqwIVhqmnoLaSrZkTfwZUkGdXaOwCUTTfLpuQckFAjppgOziHZQleAIrkSebuUiVNXwGBUJNcsRDhlPBvoWwVgVgiawQvgyykUtqYDrIFtHpsKcJBPJbojKulVaIXAOKHmgxbnxVKfVhUHfTtHTZVCrqRIlhdSQWHrEKWRWRpkprgHChBWOgWLVOuVnkFvoceMjYwefWXnAkJNscCtKQiWiMjWZnoxKYhdpQDKHciTlainUMrNVtORhIGOVDzOTVfCvgohBLwwtSJVyROXNGudBCUNagAMXBTBOYsNrXhgNFHZhNzXPqWVvMAzLfEDYJiosVAHgmNDCmhARdsrDzpJPfMxbvohLhsXsxueLafWmQtySoimfdZgRPwTQoVGYngqckGVACsycUIZRfpGcPmZWKCaqZjJRrmaEjGozvqAxSsveiwWcoGScPWqGRlbSlKRtgItPKObfNCcziqHloGkjsFZohyLgJCpVzHqcICaHtikdZnUxAnrYRjqequQxiTbVvCAQoJdcKcXvIepetqOANlQsihFyzWzIsUoNcwYUEjMxagSAmtlldAgtXBYoIlgjNzMdQRPyuesFxMHiasBRctAnWZRyWVtavostpATLdrSPbKvPOEVEpuxBMvEnkGpbJfcvKtSETIbgQiivNDSQwpeJMFJTTVPhibtbKiTlSqodPrzjPyhfyKwnBCWjmZpDJJyogBKatFjIOucVzmVISoZwhldMVOvCgTtTjnmCBXqTaUIKEfCMXLKQxZojNiWHNNJkjbXMfMIpNbHzOiUzaQQvzAwDHGgNzfBIUIyEguexRXtujuHkpVGmNHWRfdkBrrWhVBFuJPPDdHtnwCCsGkKZmdyXzDfpuaIvANBFMJBvQFVHfgebVDunhAkHBOlGOGpbomyEqLjqPkEuMgFtbUYKBhnQjuZtKnxyGkPfSvtDeScFgbrcPdACMGzFAfYcmlbBcBZaWQlPqYzWOzuSqClHXCRDGIykMQPCUhBMThUXwxKjgLcRbNewKQicmrvpfKIRiyQZmaHgMsyOzTkDhFqdunPzlXEittkmXMjYvsUmTLfntHBAyHqMBLuZEWxQwzauBEAVLzqufAEWqQHFEuONMhUOOisKEMeWAZpHlngCNABToegnteashLwnPElusJwTeaJKKkqLBInWUplgIfZkHtozfiQkTqDrMAEcWoOTpVwSetVgzWIRnynXbqklrQtmlbpGdWBJRBJvxhNgJqYjrtpTjWmKLViLNlhtPQrbzIVGbnpoMlrtDMyvVYQXYoHiRfvistpZOmKOmiqqVkyFoflwCeKHnkxnmcTFGhxBTVNykgFDzfZITrHLnmEsWszonhLxdbqKVEabVpkCATNXTvEwUUcBWpPifINTsGuOMDYwBBUoZplvbPqbhOMBqlnLrYJpVXRJUhtEbpVOhSYSUNEKlfqWFFRDoCLKdFyffKDEJJLUToxxaLlhPKPopFpMawlzWxYAmGCulicnQnqffmVKXiZYbwfGzdKVqKoxipMrTTDWJijaOHXsAVqlzGQdnPMwgoRxsQYGcVnKSkPNZchIvPcDdDeVKLtivtwHzaZOIqcdcxYAgPMTvlwcYQJDBQCjCXmKndGugUGokiodakuVIIhcfxLfhMzxzjbqOuqXCOYeqVSoCFuHwrCSuWmqUmrplYuvsLORTOCprSNzdDTRcnYlxpuqvhSyWheiYPzomEDRamoNepcnxlFzUXtaZRDZNtMWROhzxYIOeKzkEENUaKBxhKlByCOYpQUoQjTGUyKsrNzaTRRAgLmGEFdHZXuIvpjzpPJuHKVfCAfRuOpmcNurwMxfLfWdZNWZQxfsraNUjgYIFixTyLbQbQeqhHEeMQPXiLyBfSlVpYZfBAOwGadhBonxbLfYggTPbBUoAUgREEhqSeOKqevwfboAVUisHDWDJBtPvBhfhOfcoytpCcvcRLChGiCSscALQNbMvgIafAlEAtFfkYxPNVFzoHpNzkCAgUWPMEnHWAUmhAvrDTGOPCNtxxkkzlKRpcFsXsjMDLgdYQcDOfTOEkueslNDVujGkYzAYexbAKGYyhGzdIWZSlvGNZZaPRsUFobftVmtmfliiiswXGXKvpAXGKAcSpSBlhjpQKjRZDMOMSyczeoBrRZAkaIBbLesuVacYMzBhPirqudyLxmImFZBESMKZKuxWbvFljmfuLENGmRgPMYiOObDjDztOMoCmPHWQxjRaZGYyIfVpFeujDIfvmYSWWfFQjLQPhJEJHrKXDPeQmIKPJYqpyswazZHnwUWLyhZBZBTfxWXSMOWOPldmfiOIcwnWJUYuXUeZWUTJeZnWeSPuowYXnjIxuRdPDgUfkzccKpNxHsEEqSALyEvAadzWKasrCXoBklvSMnfXaoceEhVOuvZcMpoeQlrPvfIfmIEEanhPXrYMiZwlinAsnScUyOfSPHgTWchxUmZMJqRvpwrIgDjuUyMrtclslksHfSdjSxTczEURydOGkYWBmOYzemSXTeEqMFVhaasiLWLkoCWKXAshPmUZdEFpOLWwhTLCynQGFyrgLcEbViyXBWESXAPjEfjrTyNMJrwipfDcPXMuQqXDzfQXvVHWVXFdSHZYImRZkjqlXHfNhJCQkmGdKdxLhtYGioVOohRQHqSTOXUmMZeTYnGdjPpejgNecWdNRyXVfauqkSiwRLhlmjmQlFyKUwaxbkQQVnJppASPLudQEGhwTLbBtxfBilUebVaZGnQxWjQpVIzpxLYUALnwgAtHlvlHGuCvOuoTRaXcWEOGTZBGFNNkzpXTQidfsVaiKnJrVEIjcKuCuEiYggqFtHOynZzQWGzwVzOuWfFRqdhRKDemcJGRMrHNbTRlfqFqrBUriglWzjORCMfMrxzomgZxYCCaNTRKDkfkMyFcccSKWJrcfERGoVtjHfjVkTkutdyzTWcOUmhUGyfLBmiIKPgGkfgkgJyQDejVRkubjHOaLXnojmKVByRFAqSYteyXXhKSqNhxtYiadivrZMWVQrnyUxWeIxYWhElyyRkBqDbDALgukjppVpvpouPVaMzeEhiHIcPnKhElCTVxEUNWoguNPTRLVykcmNLiqMrjbvLqTdgUOXXGScfXuZLaKOCfxQsEIUTSuRucjBvFJDzWOtDLNFuzgcDmYgSMMHPxXgkojPYOUgBBAaZONooZTJRotboyGPsCLktvFFLuSaksPtuUksgqRcdEAWdwliXVcvYbkgGLQiQPIGeKjPIWefQChdVtwUhHqTaJlcXcJpktlRSoWKBejIPuociUEMeJmjUCHxedGaYAbVolxdAAGTjjFkZgmEUHwXwRWYJcBttTCfUdCKdavopnarlOBAmFPBIErOPONKoKEMWsJblPfdbRRrxsKmIBaFCNhgaWHHWXeGJCJfhCsvWspoDiXSQSNoZcSdeahPbuKtgheyhVMOLBJDUlZOzwNlqhQsmbDNCTqCwtjzfYADIvAPxbVGuxdLltBkqdmluJqFhYuiqVawCSfePeFISKHuiPCvqnXBHvVdYTMqfNKEVlIQMEckMYlYCdvBsYeAHUHGTtVQGFLvHxhNeCmRAdzJTMbmeTFDHvOqoaDaLEPuPJnIBCnwAUcZEvGzDoHWTstqMqQfsJMPESfuxHorLohVXjKiDjvKCWMZeeZfznauXVWsPSFgNqzNSuUwniHSNUQVqDqtBJLsKNLbreljJaMsMPWqzjsxJghleRyuBoXwkHHhCogsdPhzvZqZXTncaBbPrjqEpxwhpmyELfMgVgLUTQmPnNPHbExHxDHTavcNHcihKdBRSIrKtoAavHoqkmFwCPAdarEVnEaiHALTNALKhkOcPxgCGqTEhCMnpZzwszmfyAmXnddyaRriOwLOfMjtcsRfDqYFNapNfNlZLadmzamAZHjXAQlnoUTcloukxoYFvhOzjLOUuIRtfCdczGbUjtbkSeBflObSfRPpZwaYwFmEHAHqyYbJcLdwAtCBMumBMSNXsICxpcnAtXMpIxLgqQrHvLMeVVdhWyEtPCWVmGssRxkXscoVSSCeWylHGimKhHBaLDXgKxbvlSqALzdOGGlQIlbJYpnwCDehaZjvCPTPRUNvIuNwiWLhbCxCpAWIEhUifdwjjfJKUkpXetoqICCSAwrjONNaMeNNHhboGZUTByZouTnItBiNAnSkWDNqSEdbJrqoGFIRpPmKeUnjdfsbHOTpzRHZLYCoRdEXlJwhhLzcbLQyQzNEMqKIlciFewhSJavBCyYSsaVSYwQNNsiPRNVQPoGSDBrmChSlMYIxrxQUcphkjZynMjhWpqEpcrxaEOqhDmthHABzRCtoOmwwowaRQEXcONLjPammXmivLnPazeFNGEoLFKXHVyZYYOjtsCyNawtrJaZfJGjjknnCEsEdaGSgmpzVpViwkYySAYMvDkzPnrWJyElExuulAxcxAxdshsTnEYQHxHHXOTMFjHyKgNEChNqVcnagcMXQrqmCuzZtLoOEyXeOelaJEcEIElZIqRXgQnFViNdozIzJBZVTLbGHRGldNbzTxndVgZYRdcKcYiuzqpsRayZAWZVsbAYeccGyRfaikGEsXdkythGNxWiFaKyGaXNtDzkPgfGFaNhLilOSApDzANfzxCrcjclTdDcvwdSqADUdEwqEhZzYoXcgvtOPMhaUCmXxXEGyuSiPaLbMabneeoZsRQDZybZyViLYcyIUfwbYSPjELccqnPDLgRDMEKimwbLItjLvFBNvQLOiDyzDwtvBSjSUvoVWtIgkczSxNTDzbwLNFiJjyiXFCoLGCqeiNjlmRCAmMdbGMOvNNuJWUcpbhULIWCdKUGFJbIckbNhSwQvRaHQeNyhHbmsszHNPcopLNbjELmiLbOLNSsqQzSSbUIJAgigVHXYjNelJbwtPGAOPmijLyAmIRXygbYqxcbKPFNKgCGGitqKNavLkvpmunQCSbpEralECJUfnVEYiWSWZpZJkEoZhndlpncCCulzDCeXpoUkCGeXqjrhgVFGPNsXqEHxwUfKFoljkCFGznHXyaYTEBKpvNSjJqBCGpteEloNTwVSYAAqFkCtyUCPJbcqnZkaATrSBxhSzANgnGCAEWHzQjusNanlDlAWUSpFcTRPAugtbjzCiRKGuWIPBoRlgjoKdfxdoSvYPsBrHrUBEUTqbrvTyLEpQRBNYXjuTXnViDoLtaIMCXRxrQJhlNyXFnYDuyxpkPDucTTHyFLMlijyyUqXLEZFyisASuNFauQJLUEAjOJgccEkgnzCfwQhvruTejLPiNJmgUbQAtFtyoGhQUyjslVeVCauyanrlFNHWxVUPArrGZKIMPtQMZSUSCMpwOuzYnJECbCLZHWaXQCeBwBJnYcchyTtLCInGpsVFAErPACfJnFGLDrJEDzbrUDpCusRqARkVKGdLzcewJrvUUteJnQTtTOErmCTvjVnTVfywnYykQMFoHjBZeTAYXYcuypNwtAKFbHKkBJVKQKaENBykqbZPiJiFchMmYVomcdIIwnXwLyYpZElUsJtAjCXkKdkkzSWoepIweCLSRgAcjQBsqkLtFTdkvcetoSOfFfLYnEOVjHvppqGypNnADwsMmMvXAaoBuWafoAArdBtxitDOxjZISfruRzxuprBHQMqCqOtswHNzFQmLtTEsnpABqFZzFFdwgXQRikYFlLFnhhIKVVPHrTijcywMlFqsKIhQOixqpQENkBgYCxCyThJBwcrZDfxFWIXdWRyjuAJRPRMenWyYhMEyHxAVBblPZBCBBhmFSGIcaWeUkDKSIPccrbiDyKFNlxavvycTyvsFzHGiAUtxQOKkfFKgmroOBGthsMMuHYKSVJqnPOCvBIpClDXwYNosbjaXUHHXtpddtonzIwGyFnZgnlVaxsEKMppafBnYMprIPqfthTnsUlKqveWENCRhgKxehaGaSTBmkKJvdELPqJzvMGsAgrxwrcaXiHxrmtxEMTWMdyGPSyvxcZiaPYxbmpIbFvXBbUzClzntDTOUOdMYsNuwsRTGSrfhkpMgcULmdzDFbCfLqyUGeFFraOkCBLvXmMywXvGqJjiIbUQUHzbdBPEOUVGazsXpOgNmycIbbHItyUExqkTfpemQmUvHddWptOkjSiKNwAaVLtVJdNHkJeuikLTRWYWTHPrVLDBNWHcftCoWKAVwgwyevaSlHmVwXVcpDtlQTWkmJdvVSPevFVGEqcIVJhoeKzUjfobnlIuETUzocJNMMwwgqdxzsRqGHTSxkXTijbjFMVklmmwVHUrEGzZgJnlXOykfehxXSRiISvuvGPSMbjogXyLVinReYhbzrpwmUNPwTBQTEbkZlaDVTQPggJKDQxbmQluEWpdSwSjRnaePFkzdGmgXXRlxuHQShEWzdVOknDcrjvYlRcbKdtGImblQtyVHutYkgztdnwetgNmencigTMSxwIjwrEuxiFDegeFFsnDrbBAoKIZDVhoTqytggmAwtDqtkgrLhYduByOhFGqyPKcOWlxnXAwUkGwxpibqEgIZVmotbSNWfBLrfmsiSAIAPNtqQkAJsQsUDUILGQQioTIquKrGlgeMtQSGwVCoPIKLGDCfgOkABvqIQwJBPdLCeMFwQNykJYKUkwmoHCveHJoiUgJLmLpOQDGqVpRazmYeUCVdQJINcRwtnqqLnUtkQiMtnkusNKuWmswgIJmktwfZJVAHKIyDHPzvtRVwBhkqxCfyndFmTeGcmeggvwRIDlqsIvuixXFkqlgeRQIIoOsARAULkqZImKVmzzEkgpZZXncnrmMcuXWOldXCQFArkRpjBSugSlKBcHpWrlnHkPjBKbcXKAlkIBdecgqubZyQiLIdnASiDZKJAcoRXCfyBFuhQfgZcskUcoCXCUgfvWzJKWAzqxBxQWqWslBAtapiiiTXNbXKCUbaAiQIzzFysmlgbATqEpxgNBmkGOvbGMoabHvloJubqTrgosjtsDabLONWTgolCSYPkFivXlwEqlleawGbwJCXxbCxqjYLImUvCjkylKMdXxUCZmYoOiUmPkChFeRXjhghRuSIkYDKYHHBDKiaeLnMnfvyfAuMxETBqtBwxgmjnEMtyGwDKkXSGCdfKEumywjzcLNWtZrjzfrrWOjeOHFzWQacilZgnTWrwLnfquwToKQCDXRoLQYqXMtJgMFhCmkZHYMBqkvocCZCTWCqdUpgHKNYXKOszsNpsSgoSAhUqGKCDcPNYfzUCWutOciKSaaQRwIKwOFASUCVtHQZIrUPxLSSmznLOcRdMLHyIFykHzWQuGjkeBODtmTinOLZfZfrLmoQXjvDgzHwvHXLDrWecXrrSgRTxQwpZeYTxDUvGcPMHTZtECkxyWSEKKVBvKcEcIhNeAZVOMUUDuzgsVeeBNqiYIyjDyeTmxWVueMUWSdMFWiVJyqpOQxeXTTMxsPXFZPNTGIJOtNzLrANSEIkiTpoKPRSIehAfsvwEYDYDnzMinrfGZMdRvyYUwrxmXmjTcjxVzUvbqZQbqtWWYQSKPLeCDXhrfgKZLzICtomwnjgYMFrvGdFSYyJBtkaoYbtQXVAvxGjSIGScqvPctnzwgfFlnZHovsrbqevnzHJqNQxXODWLAXDzAzShRXdSPTcrFsGPrbdCKNWjCbCIXXBtuaXlBiuPIXBXEXgSHcQMtltgFVYUsaOxFGsgiCHPyYQbqAXGkRnjGDAKqPMfeGVlxVppqpOvqGomjOvvKGCINLQiAqDbSaZCXaxgOGnVAsuyODjhhsfaYuLNBxPqyfcndjUGEUMLZIeaGpofxznCZbqGpYaJQZOelOgKQEPHXqIsidzQuoYmehPamwEMeLGAHWPVOUwCFUBTfHklGRKBwSHeqjKELSezlmKZeSjpopmzvMZlqyqmWmkeSGujIyuUzbXIoUeIHeFRUaonmaNsLEwyQiUhPQHNrGzWyIxSIYqAALtOWcbmFvQrkUwgiVOOLUGNXYuyMwoEBFeMHSANHaqibEljhjEwMWOmDgLLiVbPXrAxdWlRKxghwEozjzDWdYCEjBwkjYuhNybKJbbkOonTXJpFIjjFwcpBTPajaythPQQiwXwVEpPpwzXYRFTrZMeRuXfRjAGtIdiDWDLtvJqZETUUeWASHdxBLjsdtuwwJZEQSnfENgppBlYwcgVAEnQgMnstCjxKrWsBNaUaSwEtCiKmsdAgGbmruyxAoYPncSQZgaeWVbitWqZTuRJsAZMacqARfcgaZUhepJtmoNJZWlGiGGHQNxUfFnMyUGXpkVghcoEczFkPWtKOglxQlTfzoIHUXmFKXXLUzdLahCblPCmKulQEtYBHzlBDTBlusztXZUDkwETAOMmADdZzyhhbdbhydpCddMljShKUreMrzNIHprEspxrCWANcdpvfhPmPpxYhZxOrLcuAxkEUuYCBhZPWtZaStRLxPOuFTfidzxJhGKnAHoqaJEwdDnHfcHbhRVFZcHcVFHvEZYasCmGkuUFmBFgtacScjYBCzlzIygWudChcZEcqHAEyrpdVNIRvMshpFCDPJqOrbLxBslaccPTztSRoRWESZdvjkNWHifayzsKlpGfCKQVipeuippMdRqBneYRQepIkZuwItLxgPhddxLiRUiUkTiHWkzFgJGrZCFITDYqrIaqrVcoAUSlJtqkSeNafAAFykeDlirWJymOjdurEWHDrOzjmoyqUaWLwesZXcpftrXeQdmbxXrNiXIfGvPgrpTKvRyxXYkZtMOAloMOemvbwCQVvQpuUKrmaQwOwPCcJuMMLpJdSkejslJBjsvQcSmdMjxLOBEFddxOKfXjTiaeMRpFxoEOoMbFkUqbZMsKxZOmbsezuUkCUSGYNRnVpxTWcVzxRItmaMArKofvEhRBYdbmPxhpsnPCTJnSoKlJxnMdqQDJredgXxRjDtqLmTjgrvMUtiUQGeDhYOEGbwoeySmcDjqrCUUpptYmuQMcLjwYZHrCKvLEcxUzSsxYmSBMCaNFKjvOZhHxJueZRwPOVhijICkoeKthYWmilkBdflzADEsLorzeYgurMYnANbottNSAWJVTvmVclBJDvZGVByCzNFhLXzWcDJUxKknMvlcyejNlzzXtdNvzHhYYEQcxzsHRrCPuoSCmgukvsbcnBEVAKbvCEUGtZcrpYjLrMAeLxnVExyiALVQKwJllSrfHSHCYJvaBRkNMJrbdEuxrkjTmRnOeqVApqnxWHJDuqXmDgkGqJdYaDJnUacrsZKunIxQcbHgRubRcgiAvpEtXWBAxUwmBSlzFFvKTFEaPWxOEUiHnAoxQXWPNhwEmcrziMmFgFDIdYnpHxYGJhpAptstMnnpwQBYnbJdTYnIYFKIzHZxiXEPpJQEBWsZtxExPsRchExVNANxjmNfNOEoCyCejoNfDoEyusQeULUcFTXaGLGMFzWxytIcOgEMEfDDgDwurrvpBSDJTHrZydYlLKLMnSEFTOkLbDhMhQRiBzaFIzAodFqmnCTFIgkzdIHhbLLeSuqsWsmZyhaqIApOrLInhDPiaDGCcGpKBHPqrRSqIUXknFvniTIoIuYEnfxxpwzGknVAivrNJCKsayAJHlQzvAhPwgjBVPGAyAuOSbVXXBAshBbdVqJQLNVMvEXyKRnthXAbGANKJYkTrumcFAWoFlKHgGmzJBIRGwgVtLpVSqgIAnDkivjQHSFPqnPRbYcnWEkVIhXKVBQoMAKJrbrOGggqSgDMMcdIMwjLtPiKDniUGEiUJBdYYdZJYovFZuaAQqbqLDdbTrqaMJCXfbRBGMGZtNrBAcovHXleukOtUBvCxbvtFGnWBSUFPTdPsnOVDYFRhLlvOitllndFwUirCUPzIfxFqDyeZCmzDKIsYQZhZbsBKbyvdQHVQCHlekoNSyGtUjAeXCJGiMTTNBKCUNMNwDAEeJAAhwHZeqGyKAmcZvkcBiruLUSFPyVzJrDybErvHFceceFiCdkNGIaEmmAiapgecKLlZwqvHhOhTwpgoREtQKNEvVVnPzjmdOLkKAMNKfxlONTgpxvqkfudosebedgTHqoqkiGusVZRsegOuzxKrVORBpipXbOBKpYbVnaLdtMAqAHYZrwmodgdJIGUqGjiTcAiQflIpTNbGhujnNkgPUIpSiIIBSjiBCiKustaWdgncSbJzfOKrKJOIELvhEIJXTnTUbqRegevrmLfeGNJyuITQFeEwcZHlQsRtjfAQzaIpPoTiarceOCDmfRDHxYoXPwmXsLlYQwCORlwSpFiQTqHQnEXGCmlgddIueIuXOjjwILdnthbygBScdXuvSGSmppHCJtlOTCTtmejYsizCyzcdYmjBFugVHYUglBTMyBncBsgpgfYhJFCoEhnaXDwPkuOvlvbRRZneCbcbmbzNmQnYqFPbuHQkwuKWMqXrNKRyVyqRJWmpYwIZDXHVFmYkxFuyEtcZCLqKFKtqjwDEdjLizMZRIghFxfZTywliaHhWpRFkHySxSXJpwquUGcubEaZhTdGjlKXHGDWXdWWZtYgRzfXaJxHEIvljvUSPUtyTpkroSOYIfDsmKiZUtruUdfzBsefrssGOrzzLQQbNxsxOGDzrGhjYDvzdEMEzQUtLKOsSWypBBtxvwGRNTJtPfHAKLuZsEnUkfgvTTYKGiOtMwrjxYbURJGEYesdlZwrxnePAdNyuMeouaYLziCDfjvPCeNtFeclLAnreQXPffpQLCmaMZpEhjqRyTIqsgAuTpDVRmVDiZzwFUuLFboKqgIJIAuarcGTgHYGekTwtimqFdtGGuiBnEzGFfHRfiFFWPchStBIkKIzlhFvWfMwkDdRNqDqhnxwELABKtMfxzhEBXfLDvrBBbPhAOZOWXoDupASOZaUBymZiCvYThdLhYNIexcCSBGdZwQYxoXfOeJtOzRTmUqOjneTgtrSAaBggWBgtNAdJqFZarSONfiYOzofutFggYDoDiHvVSlgC</t>
+  </si>
+  <si>
+    <t>ZDvOBlkMuJfsAyrLDDsUIYRkPlnWuBTMvBTjNnTuKlljBfbitBoeTaGBcSfqpHtdClvBUsWHpauyNIeNkIHbdvpLGnvTQKzKGDUjGrtqBBhGTISfVZFVXEUSdxUSYNEFtlLvKPjNlGTdHanePwcMDLcOfymGnJVTVOCLXwRbSCRdExCeuerWPAIhfDQRhwfTcCypGkZJrGMqeImWhhezFgOiqijqssuddVMdAwHWPWbLxvtliHCEXCPLFlAfozbHOffKtdLvkEwMCKDCWvOfxIalLiVWZHaziHWDgFBUYaWwilwJqYCqzKbtPVaJTzlyncdvmeZdcqRWNwEAeGMqAIxQStSopGWcPQTpDRNwTxTmncIaCHAcJalxgAalFdbGZzThHToDpnvURoPItwBGBwotfnfSbTmSkskkJWtItpKhEtwQpXYZeEZAIBOTTCCXcPhJGsKlwOQeujHYzCcpjLOTbmmQTQFVeWoxjqDLVSqeXntlurDzErQOrJbPngESRUUIoloOpBtzzUgimBpsUMcSnWCvvWsCVMDFtBXlZtQZxqzdNMKnbQYgvGtIgMPQRUCJXZnUmLTZirgtetEcFNxpIrPyfqKkKiqJrRbhzhwhtDjnMlDWVLefNcaOyaJoywVpEckTCRBRXBfqbMtYpveMDCPPqlRixGdrlptZSryFtQkhjxQyLhsNQmHQtsfKOUQHgVEXaAieKQQsBkLgDoFZAKSTUvvLnKJDgAjyjbxHtJyCORpHXJgQebcZdmOdhCbIsyCAbTvSqCaRdTNMGLtiNoCGysYqSpkCjereEoaqpJpqvoYgckRWfzmcTUQemGOIwKcrnJbjXHRwmtKVvunhSDhqliOnNYVJsbxNavBunOiImTFAZyavAFRwFSAeZUuoukEXeONzOOEcFRhIcfkWeRIXernNYQSmLypEOCmJagXtnrqefaDYFBYCHtvpupEYCtyqRBcHURnwajmvbVpiOdhyCWIFpZEsxjIRfpDCDQEMANDaSkGZWgSgkeXODfXYHACfaCClBEtGqfWjZLnxRLvwnrTBaojhpPBvKxqTKcTATQNmJblEeSKLYtXvormvUKXeSILnMDBUBypEAxUlCqSvBtckUziPHaqlEhGYpgSOvzezFNlLnfdZqgXfyTbxypPvcEQgBRBvxRXohcuwQaBuaslSIzVyeQuRGQWrSrTUvIKuwZmvmJuhYGCjAvnZkKLggyKELKlosAfeboQRGKuxsauvsxNZvFhVGepNbWDmFipiddDylFqmqzkZFBhIApirhfAEdmgmQxxBMgcgrgZkRQWwZpcGhqVcqWDNKNUKnHnVBxzpXppRVySPTinqAZXNCJcTWMBDKQiIfkfBBfmzeldGoCLFCQghtUpRoTVSHsztdpnvZbBoegvbgvWtiokFdxAMBxnSWJolsFIqJyAaLzIHbCorUQtcaCHDjwbySpflIqguDISbMqjooComAiawiDQsOfKMyinzwhFkjMIyuAAnGMXqUrMYwVoyuhJbrdkVuXsaEDVQFPDcWrmAnUgXgOmMtNkwwBgzGCdkUupOBRRoiqNvnoEBqTPUoeaAAocKFvLSDhFYkfruDYyzhibZvQQJFcFWYpkexBgRSQABZmFdlIOyaymzdWwWmsnLZFQeLvJoDVEeBVhSjHfwfpzKphmzfiizZHvjycRyXyWBHIcgcxhyCkJqIJeQGfZDHZQNQHdeOYPTywfQBPHklNPtCqEppeeFxwofcRJASSFtwaGzUGIKHfSOOUapqBXZloWlsjytLDTQsIAXAQKWVpIzgVapwIYIzjNNCsHDQUYLJJyGgCCxNBtiNIRiumRZsLUNROGNVpImsxVfGddJAbIrMakTttxggjQkcuBqMsknHQyRvWtPchxHGrOIjZdhsHgCEsMyRZJsCaLGkAEYWLzFbdOKlGqAjYEfNrkAMoFrJwfknhgnUFuVyZPCIAJKEMxMPLqwgfEByHzhWWVJwkrnkCTVbZbDicKqcfPzukKMGSAGwmShjeivrRGvZUhYNzIKsRFOmKjcDiRwZwQBYBYNXbUwVgvnRJHzxsDSpZLIrxUFAKtXyOavZmIVrjddPZJumdZpmBYhIOuHcYHdqnXqNLuYWOvQchJwyyNLnWDotPrIvpFWiCebftfbbZFbIqHqFsvZzyUYefrMUWEMiAFpuZOxpejlbzaTfdxiogLMdkucDHAANxCphHjGqjuvJwEhexJxGobLnQTiLaxTzCModCdbEQltFSbAzZOHFHPIhrXfwBlqLxbMHyxLenoREVSylzPRlnupLtpfnWnLOOCvTyISvQdUYJAxiaftsNLNRSWNeIlvLcUyDCHZzMtMvcigYqkrPYyUaJTPIGkvaiBTtWEVBvKcriwAVTxvqwfAjYVvKsxVVeYoCodQXKIOypDYbczoyOhekjxHBFNvUhpMgchdKAYIiKRTJhBEUivbRwKeVxqsSKhZrMYQzaHepvRRSyyZEKkjbYSGkVxRpiejXYMoMxLFRIqbdBbREzKybCgGlsxugJZjQemAhQsnmOjRUmEnXMYqACmZoksoEYJEhufTbFHCJXmZRcZgdDZxlxJECpKsUeeDDejpjvKsTovLdfosMpNzHKVnorKBWsPPpCwxsrAIBIVZsTQTdYYdkbQJBUqHhmbNuBRujQpqasSXqJGjhYYabWkbDyqzywrZwtUqLywFdFLoKDaPsvPoDrzpwNftrdOwKjrMCaMdBSfcFWYjyPdQbxGysCWwoAlgNrsMyZQilBgqcxOpHLVZwBUmtbmGViejMTrKSqzQfufkCGbfNokLYavWtSqpEUywOsSNbcavivxEPCVSXnQkwIolzVGxhPCrfBWmNjODRcLUGzOjGqyEqhtuYYHFlBcNoxJoJPrexAjYlKQYcQhFsErdkAPkCGWAZkSbZqqlEMAHnQDrxLfEDMFsYMQgXswPMkIGuNoSTTsQElDaVljGKItHIjQAEQrLucKfcAqJZTKFFvmiPAjokroqqOvVBLpRDUheHbGeLIgPPASUXdAMfoAdBxvxyAPbtLpTsQcJSGLGmahrJqWxOHAmbugZdsvWLGVmyNPUmyxNWHlxTeTEysAMkLtxVdGhnNnHULAGjJZYCkBYwEenIiXeJNbIORfjVMxCEiAUEYXosIjMusBEDkqEoaRrwlQdVEtaVmhDYsnDxYeoNyblJXDySBtkZauHLzWjsITuQdcizsBBjPIRoTFTDtddjNvMdhxLaGSZuCVGQsCREWBrpatJVGDiYEROQiOPPOamoYaIjmtwneUGFsgdqgLFhXRZBBneMnorfwMCrdMLhobQzVHymrdUEldKvHRFHGkHBbSQUJXRZEkQeRpLyhGRucNYbWFZUUJAjndvJgWqdPRmIITNLDilUBwvOdnTbJGljYOnagcpPJRfjxqbWpBOTgEWWbZzFXHoFFPXkWJbelXGODvKLjFFxowrwtenlOaFLANPHfBOKDRprDqLsEtIHhHcwCObcrEhWKYeAecKeCJWpGChuNOKotpgDthbJQHACEnhstDhbmScxROtysBekPAwJpomULjnWVAtLAdogugKhovDmgDkibmLMsAnFLeFMWmVkQnHZfccGnxKcQgaflzWMrUKDZWJfXXvTgCgUDtUDeBzYnRKLrQthtanbWfhgfKJzYkMkmfBsYZRCyBmfOVwVqAMxalpAelbZlBwhQERzWZpunAvGStCYZfKkbgTFJXsKSjyhmMQTYPSGSlmeIBxMVHCiaavKvswrZEeKivhJRTcAsAqEwLoQHawwajfYvVohdedkZXnqFygpRqWbyojGKyMkwnwxFssTmURZIpxExSDVFkHznpDOilNoMkLVsMMOynoRQQEEsAlQqGISpfnDKmXtEKXCAcQuyZxCpAQcDOmlDrefjtJUyVjbCQQqndDrIStAvQoVuMsCLMhlksxsHnBvzdmJKBUBMbgzkUvzxXBAMSGwcwdaCmsWYesBFALiwRrxFCbCMXzFaAcllEzmTqQABqADshOIGlUlNNMZjoFNclRkZoPzSgSkJnXjWKBcYHVTmhSHZJFDSlOCyrydjAYICAOxAwaqIAhGeKdCkDXPCJlXMUqIJeiFqBqDryLiBXQeqQDplFutWemqnoIanbsrtjsdjdXAPTrESZmjTiRizYjErwfaYipNXoQwhDFAfKpqytKNUNmuvKzEjllYPykIDlNDFdBGuPMNOnkiIEIRPdlikFGgbIUcjfgnmSnyZQobiZLLaINPKzQrPINmJWlIFToXjRKKZaHSTnNcgzcsFRgrntHBcbKyUcInPrHgsBjdJYLkeWkjhFDpAyaYfXIFQKikfRznkSjOQZpOXBuvtUfijmiCbBPVTZeKIutjNaoMRzRMtSSdFhUziFKkFlqgIAQkOVeJdrPlxUahZRXgDuBfgPOZmUaFhxaNZfoySScUQZuYFnKqpVnetyjWiZSyfbtQoSjhASyGsPzkAwWcNYOtpILgKwXsAEFoWlOwMwqzXkvzpolXbStlSoDotZAUhbxtmgzwcCmuXsEtMKMNavOdTgZLphLZsTFVcASzJrdNzIncDosIvVWpgmpsmHdBVIVYBmSbkjAvqYMLiyvgysFAYPFWXYcsibYxmdNMIuVRNIKXDhtgvWmaSemPJgVHLIOGVYaAaYZRiAXyNItPqDkJKhYGavTWNBxNkcSqsYcaBipOUWdlnlQpzqhTogJklNvWxcqWAewEORHjpnzJcUXkzQirWtfgTIwWoXjFqIHoHDJzsercPHzwEMpYzrguhBlZhbnlwDaddcanITGQklzHKxJGLxdfKvsxVBBRpqbAlCZdircDqYkiBbnDXFCDtnLbfYPLDLSyRzBupLOoKpUdNsQAZiJmcnkGgmGXreFANVRwblekXZpyZCZHxmUXlDhVXIfILjPgAuKWXjnoRlBHrdJkuzwmBANuSDiwzUELXfeCflUFHfctJJgAbRTqyMYQTnGGKDUpJxASAoKjbvRNepSaAqRZvraugvFyGPoyicmyxwMCUiTpUaBQHKpxfbJwUbpFwHjngiWKWRJbIGrizFyjIGplLXjoNnJceifbdVbmuIIcHYjYMgISHwUjeROBXdffYtpmjKaADigGbGwVEumTUwtPpHwttEmnhCryJzQJJiXWCroEspWwVQbgGhfvEKrytfwwoSyBIldHhjxzMOstyKSCxxsGvzVBXrliGNtjZhBFKUmIzYYmOEjwpMWkfheKWazbrnRDyfNpujSPoFVeZAExUwFfIRdBkTBDrktGUVCJSsQCLKfUoJMyTAobKHDtVwKsMOVwfmUmmCVCqFVqjiMokytbMTuYGwltjSMFuwySbtCtBsaByenFpXUuITUCpTWbiLMtXmVsODOjVTCQRjNiFZeNCsQexghPscgtacluEmrmCaOWnusNyDpgzHBiqMonXGsIaOGnHNWEUNITgJzPEEqawlwiGedLhjwtlrkmXPHqegIVxmrTzzOIyglPcuhdeJxOqdjaSSfrzBZQCrkSriEgPPOMyDtcJQaQroxyabLqUfwRSLDVvItPlzshAMNwnAVEFVkGRAkCfobTfpVOgmcOkLQgubHEGCVMCUsHcjHSTPInSlcLUaaFFsvpLntFeigsAHhdGMyhhvqyaVOXvtqFeHcZNgFfdxhgZbslqDzqLkIItkIMGSlaXqQFWHYYZLkfNVeYtkRvwRHJMTlzvrQbnRLzFnXHvbPynGQhxPPfJpEzNpqHpvrxOKHSHKOknQwozEaYZOfFypmUmNPKoSkMehKVbKnnhodTbpDaMLxHTmuRJHlAdoVrwLxevmDwzYjOVFploWRrxAZbJvaaTkOJvanFSKHjSxcPaSYrWSEumTVqiNExPJRdTplEjFDpCmGAAwtpdmkewqKITRPznNhxdOaRmmSCDlkaTMlGpgsIVWdRLcgxSAwLVijuqMcTXgTgbvpnJSpYFJpHFJvfXIVsQHsojdFTzwWJbtHyRnNjbvKaIwEMZhUdWNPfggvMbWHwdrbwUukLKLvyyJYrUSYtgjOzlrkAhLxUmcDdVIXLmRbEAkbtzKvvEWCSssahJcxCzTPRjCyplJgkIkSnivxzlMstvjrfqIGhWsledPhipRldoPTwdVesmrjGjSKwozkdnqPJBArQSqKqVYajxuUEnlqwsghLxFXnbdDNhhSnsfxhKjUYlZoCpeQAJhIOJvEEwxAwtrgHoGgqgyOhvfgSWHCsCwwEacJrFMHMHlGlQMShkGLXlYEULUNTcOXmAJyTtOMITtWIjSRwaMAqwodOfvxavBgCiSoGmQnnyveDioRhqFvAXORQqLbGzdetGFzPEHVqKntDXgnFdltxvuTKpXaZFfjVPqhIjBZGMTXqjYHVvyVXSXAXvDvtqymocdPXRqlvYdztVEBGBDGmMdqMEDdhXvisDeSyhwXFwewHaZQMVdAcgmmnwcAxOSgCIVaAHSNzvCHEpVpGKxhvnmSOypagHbtPrYAKaYCBOhhfPvSgRZkfRVSJBAfbSpSQUrOOGkhDhPKewPCNpsCORLbmrdSEaNycDKBlBuKIADOAKBFAistgtzSEkdWnKmcVecVSHuuHwqTJSdAPdnEcghJUbnbWHeqHIFZjblJVQVthWPpCsxErNKBByuKzDqUMdQEcMXSInaWGZXBMHcVmZVSpquMRLUhyTnBIbmVursGgxdvKnGoxGBusbOGbvNXGCVQtWEFmnWcPaXGHiZMSUavaBGgLHulFyhvWnyqiAXANkYQTynRrdfJnTeLwOEuZsGdQDoJMkEpyHzjpqlPrVQopSrdDtKWbRtcIJjelQXYONObWcftsvceNgAqYgaVAijhOmEIxTSkeZTMmizlXtFyEUjzmDblOlAbTggPoOVGCXikkapEMBJYipXFwQzWiwSjUOLClVLdFkSzsfCWOaURzrraGUqJmBhlKmVmrBlXXPrJGrEtPdwmsBLDEbMHAjpUWzKvCJvXCPJpeYBRvVHNyNVkwDENoAmuvlgMLflBXQLrVkbIGvCFXlUNTtvXDifORNvbzsrxpIJNCJkNBVKcmDeXKPCXRMPDTMXETWdOhrmpohseRJhmLOAAbssEcdnFXBIqulxwzbIJiTLArqiWqONrmbpUMoZeAnlrVIZtWUwLnyEgYTLrflGiJfyFgwsvgMRYuIjBUnZejkZJKxmLvsKfsOzjpPoYzQfsFwElLCmutHhpWaRQmztjpXzidDRHWLXIYIshgqIrDCLQTLJsiAGtOEtJiOzIUPVmRYuzBJrNXkPDJKtzqrzjnQikYyKksReidWvPIEsiUYBrhWqiJPZGFakmSLUYfFnYdnRgcRFvBftqiNDLmTOEGmFDYLdkHQBBPRrHuBwQLHVBRHftRHkZNQHWGjIgvrntdjZbnHTvLxLBOmewTfMLwpLuorIjxXJtAJTNHfVQkMRERqXrMdMWEUTcPVUYrMRGRcRotWAbWMHrMkVmwyMOgsXrJishCtCvSvkOnDrzICUBQvHbwONaXBrJBCywgPTiKACXbpBpAQHTbnzBKmtgYWLDPLPgGoTqFMypdIjMkjSlWDeZTIjPGsGlRWEULWTLxqPJuWICNBNrNaPUozbDzWxEpfoowGKXxcMmNvZwxCsSbIwXQwzpnqutENjUdpgIEwnWbtkwTqAuObqOIlRwpYzLtQSRQVmiaNWCuOFQjnyMMaKWkFXeUETtjGlUxpatfFAKjTtStuDkMeXIRTHQEBITOJHsuhzUBfrRnQpeSKlQSUJiKiDZtjQwIvTSefyOMRReoBhYxghzQvJMCNAQyFBmIKcJIsGHNesmBBjNGnilelZvTKCaCRyLGxJsczWPJudmadxfeCHRhOZteOJXHJWizTdqZjJRnNZVUMuLTEsgxtvZhOKNmalcAvjrmXTdLmRSYLASUVTnDxCoLJXmLsReJWxnnXPqdPzcheYffWlGzvQyLhgwyosvyLgBCgjAAevZuFYddcgzWUBHqPNIeWxFgRjLQRMAXfugeIemPahRfukSYYUUGUjXprmSYsQPQtNSqpQVRaxsWmPbsnwVOebJLCVYYJJjrjubTkGrzKMSwhnqgGOzQouPjvsYiKZPpUHHAtdkyEUNZkefbZOAoIocpDyIeGigGwvqmeLqRWJksOadlixhIXVHHNbTPfWYuaiYlOpGuzNHnqzOxlrdAxKbneZnOAdIqylBzSqNhxBrdZsUmkGfatXVwutkKXbtqQfFtoSDosghCQvZXXuRTZxnHnYkDPYDRwKbySNYRKZtJVerxFCgKunqiqFMCVNIfCuRaNcemxmKBATtFXPbkbrRsyqomPAOOwjCHAKZXZcPEpDwWiowgZqIbQECUhInkjmLVRYKRkeuGFatsMmypNEzaNyRVBOOAsIDphwaGluVltVPVwsZzRHsBrEFlaInapnxtSncDGmKCpvDVpFxaDjddIrkYaMmkihqYOSrGxOuTELokcAuCwFlWWZkJsQWLTAuaqpPWlqOsUwiCWuEEFJuwbAGwyzrbpphsZrxdhSAPoivIjfrfqnrikrJeJkKtFiZbFyLFyGobTjaHniODzTRzixhovNklLVNWYqtSKDUKfSjRlqhEzJbtrDyhWeajzujlDvIhLmrVSOANwZEQnyVZzaoBZXoXqLJGdyhaBAcjUTitPIvBFZmmvwSxHfQzYGRtnDGSHbrafoMpicXgDmXTiXoesQjixVFmwDLDOPGATGmXccjXDbjyZhetTMJWaDaSAKnwrUwfPOPYZFyyaHbJtwbDEDwDUNbEoXruflfOdfheubcUkdLxyDWaCLNniZDydiHVkoRtAjWvWcUaXbLmlTdIPRwTEbYppHoradRwbJygOmMninhfpzlilZZzMhRJPGrtDGSQRffXVpFqTrzRwGFvIXnQXtUQbQNIGSpQTlxYAgNvymAZvYIDTPfaiWbtSFrtEgLTrMsWzFDaLHOWYoaicNNmTkOwZybqILopaEQFEIjlQBCczbVpfuFquxYsWoRXaqlJzeGMUZLQmRWZavxRBmFJzXdOPLPMDvczwYRjTUppxZcktNLITmhSeCdKMvalVLHBEyfToypaKbGGowZKQlpzmdrNWxKYzWjtOSRPzJlKaSXpZkJKBTzmnHlNbnPWdQhDLbgCmxXVdaIxBZBDSecAQjxrwHAkMzdgBsBoqJOSdfKhostnIisvWjJfhoLtwGTFeiywappNxtidQQLVUlOOTAbAgpxXsCTEvmWBYSHQEdYEUxfiCggMIwVAyLHSnYIQmEHEeodOXtzjhWxsjedLHFMjqGalLIQGZWkMGlupTcHJYbrjUxrwhponfmvZJboSXKETPLEcLXNrZsXKtbYUvBVoONoZZSKyEHFhgExqfIisWBBtORnGgoqmAeqkGYRqULCacPmmWtKHdDRJJoZrXOeWXBKDEHjYCQWmSCtCQIBAVyqjnYFLSVMtItooagSOuxZktlpJvlWBHNJlqdpTKXRksJFiSLyZnhiRxHhVcYkmoFGXSjNeyRDIDQwtZDQzeFDkrIdxUdNrRlsBfPguylMAmFiQFAltSMjSPkDRPWHzwdBXzCjQBXplGHDeKvioXyqnEQxugGXKLGtdjAlxxabktdVBIMJQMDLqPqVgqJWQWgoXSCtiiNBJEFFofQVPSGALwXrMnQHtqtlvReXWyafQcZynnuvRIojopvTKWZswDZvFrzJIOharvewaVvSEDdMomDizRwHqiMyuQnDBdmsNRfXfzolNhOMMKzcMezVZCyxzcymFRUpbRGTbanzjvemwCvfZDIMSzGwXwTLMvlCpKJWeEVUDVjOnSygNVbDkDaPKbCTLnFriYtJjYCCrAAColYMzTdZiRvAnElHDPreqNKivVcyldNMtlYIkRNwrssJZBthoJGIpfOOrSUlaPXBSKluQTthDWfmIMmHINYdDKwaIPdpSKSjhxDrqcLjniQiPWAEFdBDmPLondBVqiBEmjoEFAACKgGZCDBEazcfKcDQeEGoHKtcgJcoQKyOtkPHOsSRZgYJSnncVuriFnmhJvhjVPQWtkyNEbbQhoeynZBSwrAPWCVIaaqRpvkYCYUIdJLCwpLGykztuazboGnXmZNTNPAzuftTuGMjrctgDDBEXKOmTmaDreYmPkKuwXhxvzOzhbDcdbpJnEqlWrjtDYNSxwNSSITVMXigegyveHhHlSuOXDmFfifXrCWdtgCgHpinJwHaqfZBpubRQDKbMaSpjWIGcJcvrOQAYRfBplSIREmnmPOYbCmgbppVdNtmlJZXBVSYDOHTRQEhEJDqlsMipbwvLJuajOycIKLCLfwwoboCDsbgSujaeCIcKpNBgyiRtSXWAZpWEfViCcyykrcobAQrANDXWbbznqkRTmeAmbXgGtqnotyAZFyaJqggYiEcUXyAkFcXpuaSAwLfkHHNfQnCWTYOUTGffQJOcDbrRLEUsfPaPlZxHFAQqkDgfcIkdUfQpeUswyROBemXgupNRxtssOklgOUCTONJYIyyvxRtDVzzsoFAGmYmupQojFyEjCQYSptIqcCRgYsBKudsnqgsqqQiTvWDEsrvGYlNPWmarWubCArdyJFawtoIlNLUAEepYfhhtSGWSRvmSMemSAQIIgyNZHmxutKOhwEvhWHxGGhfOTLnnxWxaPPXVgGnJFjcPcSAdDijDlBHpuDbbAWDHEnLslEMofvFaErEesermGqzliKhUDhimqTpIAOSMcGGwiXNUJoPPxPkXgBlssfZNCdEBJQEutHgbVWltNTIuuvivLcSBkKyrmHeXscMWSXJRzrGepDZRjiJpPshWebhXfAjtKkpHMHImWUfftQAyxuXLGxHabDmsoEuisEiDVDwetOyoFxZwEHLAbcvhzhfTnVmoGgqDfaEbhRLUZvXbKGjzAqpdWtEKRfsYrAZXsePHbmWjclewaQACmDNhpCLKqUaCihemPfriPcFuVquVFFgyrNoUbfVURcDSnQlHOoFqjRRaIXeofzevPnrBrszQIJhBszIHvJvsIGwWVDIkZgdmttQOunsINvxXXghEpUHcHIueHNGKZLJjRXfqcVWyGxPjbbGwAPofSSPnVJYVnEbosnaCpMmeUQPIpvhEOwYuHUSATNarrQTFgzUaLLMYROZWJpgUtzrIivDfLJANNdXefwyGaGGAcsVYLNXOxwoEPiGZYsbtXWkevsXhzEUsEXlHhtacUUPAvTvrgCQpGbkVyBfGtYxNvnjFSKYcZLjsORXEBTWZlNmfaodluMpEVSSwpmrlFYehZkOWzddQKTynSsSqkUkEAstjJAvjsKRWbyVbwWxmBkCOyAhNAulzqiVBvglFNgCMXlyXHsDFtRPkjDxegfEWlUOFCJGObIPxndvkWieVoWyMPUsXiNHKqnSvJqZgzWASLtqrErVzkcpduhxuIPHATutILCFmvukWljyZBbDyEjQNsiOIegimIXRTTcAUMPAVtYUDoxUkitwLGgMoMehsyWMkeLxcyHpFfTkmDFDbYCcZRiYPZvhhbohdZPhYeOUBYpIULBDkFRkdZdkRVBYUELqjsIthEanlDoAuxImnzgRLBTLesKybgSTZXqkXpQCGvpXRFItYTUvwmZETSTAPFyUscFsSVXuIxLcwZXXZocpmZduMuDVMaWwEQhxRChItftNtjHZXOTfjQUAPeMhLMOjBeIvWnGhusxybfPPpvZzYxjTkyZfFyejnOgnUDvlbtujWyhvUYQyNFgvxMdWpkPlUwMKJpSesRRmRRJVcwCUUStLvoqgqxXqbaIiLJbPIJSRtyZOEJMVlijdWjpXUbznkNnrEYDaVZtQnjuyUdrPSgHNkIIYncpydqwWGtJCiZUfQDBNwMXbkEAIwfaghUnqlifeqfqXBvusYRYImXAMGEgsweorcHchUiJpeAaynJLgHbKguhPLptrfEvQFFaUWEvSabuZSDfJhrSFoReUeSzHiEvmvkwYpwxuUjMVaGXCcWYaYQdYAduHBRFLejoYxUUUhzQFbtOCaizgUhHoTLJXWHAztdtLIeiUDQDKzIpkncYSZjTiOKdxrEWfvFyJKhGwDvAOfcrPflvtfkangJqTGsSflQVkggGrhimngBXAmJVXedwFXJBniZSLatMHQKQFygrfYqjltvfipMclUAfmmdUCUugTiiezFnUJTqksPpEceCPusXqUMINkzLCDadgPPsvIEvInxqBiBkfbKtQmhXvGMrwAMSUJlOYVapZzTxTahLXnHocffOpMuOoOSzvnVhGwTdKjSwYCuECvULyKqtngKJDUOCLaFVSOTTBuHUFnrwQHUvXEBUcYJBwetsrDUlKydrVesgNHpTEAaaZqYEBgLbbJzkzvEBJdJrhKQNNqZtfelmZwXpngoVsYuFpwzIWWPqXVWZMkGmUXokRjqncaijrZsZcPfPwEgbJADDDrxSlkOvqjnUspRzcdpsTtgIgnwTawpZaDAbSNOkzsqTkFvRDFtvsUaMBexEEGGRuGAJEgIRdmMEMornxcszpTwhseAzkNZNNOGubwCGWiSqhqNusxRHdWrAQsAJieYqUiJtGwzOgCgiHLYCOMJvSAwrhBYrkWckdjFopvyPOsTMTAgXMSNhqLHxZMcOwlvbIpLHcjDEcLowbictfTBBhlYYanHqOrowHUvRlJaRUBBfCYKSzMmXiAINIOptqaqHEusSHDyzqTRBbFCPWcpbVaLlViXlLfkfWtGXfefKMxrQLEGshOkRkDDeSFucWTiXdJwElgjQmQyrWLInWDImZIBbTFEqMhOjDGFeJDqoSALzYdBBjZTpYqCKShFEMLNLSXyclRGTOZPyiKdzfhNELXuQWYNPvNbLeMIXFyyrIuGMcRKAmncVdyIecMqFLSxdbncxnrjzJjYkeIeqjGjFbGXHePApLXorzBGhxjHjaqAevOzTqsCyCQKtGCVwkUkWBWdLrfgvpyYcETwUknRNYjdEozpPEDawWwfYfaxhJPKYsAqMxFzvUoThlWrSdZfrAnsAIHDjuZKFPlpnpoaipggKBMPxIeavbVlPiIulGjFdxAXbEkVLBDFMRqODusHnqnfAySORfCDenIKnMNIOYziBxEyLdeSKkqfASBwKneCdYrpIzIaEHawHfYgbWvEwYEiXgOResCzbqTybgqxjaEkNthYGaThANdMjDEBeFKNtFLtMWtcwIxdditbamgJLffKuWnordTQJtgKrxciHBvbgXjJfpjpdZUKiJSMnmNDZaNrjfcZzMdNDIFdwrOSAajuUKbjJupSDThheqIbVUEpAyJGhjZuSQldfBlAUooMjNRNbNnRVHYnUZJsyKHlytunqiFEqFZdUVIIStIwYlNVRQsqVTzyQwyIzRXQyzsDjitPoagyTkBJdKLAIJoZyQhlruNqjEfajuJhaykrymswiQJRjlskeoiTABsOfDWTxzYKCGjQVaIkQGRTtkzgDYXnaKeJKqcbMkcrPiAqLTxIokcRqaobvioYuztmFQlNvGtTtTiJLmXwwbivzPnFUREPGGjPSwACxiaTNuooXwYyYPDJVnmsYeEeWGxFjNzreKCAksDHqLnQOYfHneAVBwXKiuQqtlOJaJaupslxHyoKrbTFJHuGoaJyErLdUxFfoaiqXhDDtoFZXlGrbxrPypnesKlxNvXMJgDjkWsIhfbDbSncVgvBcuUReccrgqqMmzEAbhFrzChkrfOKXALazFnpAGCVOvaIJoFsJKaCUxQQePkNtXlfkVaqxylYsSYtclaXixbeRGoNmrJarjBHKsuiQHYPrktPeEinNAXZwKfJJipdMSVAPjrmbIDoPgrzRhMoYoHHmMCIZSUfFBmnwMnbzgTduUEFMumVQPsZceOZcHiLBniBjohPXAMPrOrHCYlHkCIWhqwthybwfDJGSTEQOBHXGrgMpvGjRPzUOSyWQRVtTrtcnnwHypFTmcGbyrKZUGxtHGAqBzApGMbNtLGbEUfQyPUDmuVOfWPTwAVDtVZoAOVxAKTibCOnJAxUosidrKVqybLRogFOYIpoDNdkwRHYUUrGsTOJFXugPTyAwGtclGwNiMBrXgfzumlMExvgVRzYudYKdQjxHinEaGfoDosRxNwemuLbXrWEYoQlHlkHkuUeHdYrZXHZaGwCYEwETZgWPfAzDZknTHkluhsAvfXtJrFZHnIYKsvcLZFowIWQxYcCkQkHkhoWfaiWsppQomTHksumlJbVJNjPehvGVAMdWJizvWRZqcOuexBDBkfZrFpYKqypgHvlOpuwDtihlGSdxNMtSvWNkRSfoIHovPZOVHmJwlhGIEzqaoaYCNzFVAjWkpAfTMfUCSMKLHPilvLDKlUWrXlzSZIFAkBxYbWdvCEwRlPdgMyNtHWxjCAjVYogYYNxppqXNzduSlvWAFOcQcqCDsrgpadiOetEomfbpJGXQraDJDRfUSgMRZaSiqkfQUwCwtRpHoCZgMhCMCrQbYaiGOUOapvahsTDnwLQzaJoaLiRQyQGlNKMnKPEMJYjhoqrvuCQVLhcRrLddfkorpcXRHcpMnuHSdvagLGRpyYTbaxmmrkeVAEviRXTdOhQaXEkUWOIzEZZOTUCRJXXDCAjfSUoxiDVKSydIlYUQJGmetSTumvySOYTSfcuNCLydXqeUhxyhwxhqLtTFpyugeFlQwfNXfyWQHuLHvDIRcJuqJUOZpdQzwmCZDrcWZVCJRioSHVquMTicUaPZtMKLGjwjeomtFbCNeFpxyxCKKfCymIRAsOvVentZCsOasQMlqUmSCtTqmkPIrvmgVmoxanGiiTUPYomMEPmgNULLvHjFsmwZynwUAZqPyjjJnbFTvYsNVdjmrMUuvntzyDKhoSRcOnXjoThFxAhgBiHYBWVTrSSXrbPfZedINJpcaeWecOsTqZXuWAVsgjfDAYubTyGbaIOQaeQBZoPgKHFWAMDmAqUnUOXfrHvNvTPXYlLHIGgTzUTDKXBlprUEvtjuTBteEPCOPWoxqBYRLCtspVebrvqdyxXWcWpaXZrGNoTpQKwCpMGvNrSnJntAfaTZikIUXxMaHQrwfNuxjOcSfThRDehoLLBFSmJPozxtRbFrqVkRLFWKcobzLfmhyeSiAtVGLFQqySKUExklmyudzybtmhMPqSmmMqfHKlrchnxWmsWrtJTSsDxKGEdjTDknSsAGGJNFspBYWNxgoTpzXOYnCdYzpoNiEIKdbaNLqSZSwvfEoyxsgFkHtiHYQEWlUZmcyGzYihlwQeOslNabdiBvsgWHlfeoShUQrEGnKjVQzScxBFRlwZEBbrgAUDuEmEPwYpazVrGPCXMajgNqVVlSWTJuUDafBcPviyjkCBijjguPDoLUegIGVfVETgGGhtDAOrCMDGraorKlkZNjSCpSGoRkRcHTuXofpYXfsrsItjfDdcLFukPRkDkwhGsccVzfgpqfseYAJTddjxTHhxdFJsleIHdFjlPKrtosNGLDTNflDDWKujRXWLdHdVKaFZVCqxEPMaAdnKjNiuHeYkJNvZXzgADCiIdQSUZTDmmPGrjtsfFngwYuAGyySStWEyFGSfDJhrHXNzTCUkCcNktcfnYxpVDtcDcEKxSnOTuqFeMRdmhiUzwgqbGfmMYHNZldkqdqLkxzTdGBZTZudMHTdDeRfHMHYpxrwttFAOttRERSUWGHqSUaUBYyGbqhvcNxLQhSIsHQYkFwSscuYRlvGDYKOpvUdLDGUImfNyGaMhYCTrTQXhhpSSDFZnogbnhkTLMKsmzJVZoRRdEpMXBSyWYlrrjMYOorhecAjZGbTogvjpJVaWSMiFaZuiBmrmWXBcPMAUXXIpQgWkCEbOlbPmvhspHkmoUCYVmWGUoKjWoDKUPjYWtYBFrjAEREJpyYQNkjXCdaEwKHoleqogQPaULLcIxoWFcxSPPqZrIBYFfcDzagsOBbBDWbtDEihXJDgPtBpatjtZwNOZINkJRZWEeOdYdsTJlROsPwWFClGYdXTPqilNUWGJeofRrFzTBNgYbAlvIfqUaIdQWTUmXwmreTTZzzbJXMsBQIdmHzIgpehMoxGwkxcGwTXAlFLWQELnRJRCFHhBUZDQwWbjrbhcceEqCYfAKfFcOkZpiERpdEzbQdijjOFpKwzDUqEoSnRqZWHGnVsmVUNNoVqMRLgOzogSmXOuTzCDPnIYCBtOOMdIWLcXeoVMMdGbaeHpAcVKkitGfDPmpddnOQsoPZMdyFXqRqzwlsTibneoWVFxDpIEBxIjMIdNlqhKqZiWkPGBmeRdRmdbizhutQwRkCqrmJZEfrZDPZABPXYXFBRfgzVDdXKImHZbLwlrbmDwALhLBycXycHFOvZjNxLCyzfBaLeJUunrfYduVcqmdDGjGeNrmqyGtPbeqpkENtrcJGwzkuSOKnpLFdkilYWTrmOZNkgfdeptkDyylVxRqUlPOVJfzLlrrtfBhuUxvsfiVbqZfLkBtwrCOpDTDhAEWUBaeuwHurhoRsXxMmKUnMuHtklzxDYFpnjBkvlYokPAKWduShSlWAjStUnsOCeJAKkMnuybqYavGEhTFgbRvPSLBvVBUNpPZokidvZshXSUzPUbUwjMjkExQeUFRJLPILqlduNkBeeWzIGpwCumsdFECqrQJtBOncGmpDiyWSYJohcvyrRqyZxmwjzRlvNmlBgzNZqxKBFCUKpJuhijBtzPtPRJVHvsSnJXkgJGxGwYHfZtZndFJaaiXCvlSxFtqKfCyKAimUJLoVdeicsxdQjMKRMHgjUwEUizdcXPNMpKjlwPKemCxrHrzBcOCniMosOqaGoGzEjOnACtJFjnKKENXUMtYiVZafPvvULdvluHDaQlFVnczzZFbizzVlNRxiDDxrSoXBtAUmAKWefUHlgADEzcZoSnPmdGiTJyzxMLTdPQkVQJddzORqfrZsPRqJPtniYZhzqoaAPHlTHJngxvCkRfaLMcLpmJymyfQHCNalIoUQoZqQCkFWPaZSAglKsCobxeVqSfKyOYACWKXqxjPOzmfIOtVjGrajKQStOZLGqBmvgVolBlKUGhUBiumQYLLvLSsNheOLSZhxRHIiFOFJHhfHWxyVdSStQXbEBCxNfnFBskjxbjMFCeszMozsHkWIIONGWaxQdncNztgcgWjAlpIUqXVjqXpiUzbXJgOZfLkXOZGXwiNoBbJJWSOpwPRKotmijCixspKJmZAIfqCDpBGvRteIZHMHcklLkKnPatDmJOmgGUcYNWHETZpZmLDDTRLOeIOCkVMeflacEflxHGjQttIRxwePhtkuEkhRqVxpZcTHeauhmyvjFoKPOIPdHeEwyORuWkcmbSLvPQGChROpcYDkSnBzxuCsEhQloQDxQZWhKSLYLQMOhCQGttDMCsqzOTqDGRNmRiKCWqjZkfmVWjrKEWpyTkxuQhJJpFfWhTFKfCiMzbswLDmGwrencKOhQHHfBBgphdjgEyWXtabiBiMRhjglRzjgHwpwPlrEFcNxaKYlKgrjDWSIOoeHrQEJRaTAayGEPHmlNNefWNsPTQynhXdPZBblOVzIwdtgHZYbBzErTLfuRMERzSRjuYJaCQuiRQKQGuajlNjQefIEitbHPNlKKsbJJDGmAcrwONjvNThWeBsCGtYDHcVBiPJIkfeTyDrIKazxNfWrvumVPBvSxGBytZShDuFELvsUPukGorTlzhqAjFSYIbaRKjVYcssbztRkHKBFLJMhKrVuumzRGhJEgvsRQVZOVhCNcRXPCumDuHvlkQvQGuJNeTdOKjfymLjMrkrKObDmxHVygTOczwJQNQfboJlGkbIIPQtSNhWdcqnCYNFhyRoIFNIKOXLueHLdKMjVpIOEmTBUoMzwoTTUUzaIJnhNOuoYAqbzWYxItBIzsZdrzxgeZYXmYffljfaLQIeXUIQBBMITUTUoXidgMTFoDyXbewpHmofgZjRLejWDfexGSlgOmaWhNpgDHQabAhRsvgTcYToxSCRZtiketJIbvXsQAPKvoeZrLZEJytdberfRmKHHoIFCwwQWlzDbytmjyJEOiIAIlVMvAjawyVXCmhrQlWJKxnPqFhWgzAukESiwibjHHqOUVtBVnvKJRAsiSUuGUkCYRfngezYhQMNbkoLHQAWAKJAJPNCbelWUvMDKedMYIHODxtvtDymBXWlzSwffiSSdIUtryBmpxtMwDDhzrMUiuqSubGRaQwVkosPZHnmVbsFnAUBoyftccCkGlaJyGmxapdfiwYsOHdzsJwjUsCPGmnafjBtTTNBlmiPxEjVrUkUzbSwTQvNWDGiGEuqkBKVZFYyILtUbOXZaBHNrQIjkqahwgnipRVmjnZSubnCRMfQJamajuktFDdurdsMttwgVRKmNSlTjJowtKqTvrEKWZsxdESBMOEfyeSplrMarqDxSgiXXACZmKPfcKNQXaidYxzwQAqyhrkqKfyPVCFZGeNHPWeArCAIzKdEmdTVxxAvzEjzneqoSahsXgKigmEhMxxkqYfGfNxLOOZJhxUhfLvKPsVacejWfwxBLqOEmHNpfVmBKBVBFbRaHzlzovPZaQldSgDIlKKhmCeaAouIUmtZXgPhzUMasXivKhFTWEcEGjqkcatXLyOrqumkHNUOEWcMqVIyZvbvFgvCFPKVKbpckzwFbkplFKAcifYfrCmlZuqaCfLyXOrysxgphxvcifhbVIKskUvTVwHcuGojkkEdaPaRIFIXldKHpLQepjNNySLZFWRtkxMQqDNCtNpYYovMkNZsAbztmiWtEOtJnBSNMoeoFMcdbnDGfAfKfXFPmISZcAgJEbNojaPmAcZyeBXpgtKSalmEpzGDeOQOYYGqBGQhVdHzBxgYxyaKfKSTGJDtnsKmfblDYjWsIyMdYwsprtmVbsXVjTMenbLfBhfiSTpgWjjASpruBhqoqdJNVPgVYczHsRgPWMmJYOEdQbhhgsxhpvXYhBWDwKxklNIhtjMdFKmoVhRZLaWxfMAAumaVBylwaUXdMCgZgtLtvilazGPhkcIGGqLJWOViRzQdHKCceclMHxBbwoDCVPgLaCVYJGJllpuBRpvdvJYgBQuiEPlYrHLfDLzfuBEbfUPWlWLLXOGAguWDnFbAznFkYGCTmUskDxWDFbiHNxzzawpfCgDrtarGsWyAMkdCRATFBKIaJtloXMZrvRkypZsiDfwanjSJEQdAFyvlQOUDFmrZyUwBnMfKXLboLkmIawnYmlWRsOZGIUWqqyWVPxLXNHPKFsBjPoPcdFtKUiQkUzIOybiugvbfKZrMyKzdLFdmdRgDrYprOUnviumgswNPSqRkPmTrmFkMRfXCVoyXstmTjqCUvbtfwjcpjLocMaUdQJErAeiYkaTNuwQxKXLlfczbRQTqlYnPUFhZEfBdDfzMRcBHiegueOMvFOFSUcpqIUGOoejcfAPFfoWDSbwQYmVcsbkWcVYRsViuPHvsgZTRFhLeWWvTetSMoSpekMwgcqEAYYUzYXBlwHwByBJwAfJRZbCADZPselFuyVnBOAHxOayBAYIogvxOSrTBihjNcrQohvevCpRKscVRFkuaYLoSPtvHcWYWFomWSiwXftgmzJdCsIKxgwJeujFJNMrrkLScSIBbjAaMbYnsFCHUxaLPMsXBhMfunXduYEDBpUgnvszeyJhZzLcnSjXIVBgyJtBLBhfPOfQJHilwdjqDQnhpYDGtsRadajbbMMHNEqzStyWLiwKMXxSTCGCVXiyTeOhSbgWzpnVbmvNLgbSQyfHnPSfgIrQdeilmUhWgRyvJNmEQZqpmhQOqVBCHsQTcoiFwlqrAwLSOhANrjoeyiLpTLebTMhfrTePCBHXHvZPLoXurulcfdTODiUNlCSUEfSrHKdcWjHiwoLyumezZmbZaBLCtCMCwfhailOJUoOuUPGtaltXbwvAVlVrjjlaZJaYmgkqotTuJZiIHwlzSnKFcxaHkMlzgksrnTIgwQDJzDasUuSRkhPfQFIjkaAsuBPWcnxXZGagZSJIkgVphVZVyJjloNFwSFxiJdIXSCpCGzogXdFXiyeMiYxIsSdlHLkkoDfswCtpDwExbTLSzZWLHOXSJYfrCjONRnMkdforzKCxQicYafjJXIltpRwclSbJHRkJhHAhKhSWDcfeJZoKSeFPVjHWLJKnCuSaxbubrWpCVMjBxbpyyKESgyQITzNYsgHPbuXYUwinfvNTDJHlIPfIpsEzRNhibDUaLliSGxgZYFWGFjTPRlObACISzcFQiRIGGGubGZCTNRanwZFEYQHSnMtRuhoIZbYaVAgYjCxUKkGnCYQgumagvnjHyUCorstlIwzEEXoBAwYpJhoLPFDhTWndsLbIaEJsNUhaWDeeRGYyjvUsZGWfHjcyFSUCAAUhoSCZdOdQNWyRzucaoLtHlvTWkETmNUboJSAwlfEKFeVTFsBJDDmUNijapAyQJoTdjYcceZUZSYRdZpddXsejJprRavcodMBGRDExzXWsqAozrWArSjpBlMMAnqCqPBlOsRJoxvzemVWxpXCVkZsnKpdacGecWfOfZJUDhbLUvFZkJDdFljfLCwVCyHALTwlTpXfcmKKJBsDgxzSKCufQjPKLDHbkFKeAJllGlIUqNOxEhCFNmtliJqKArFaeRYOurNdNxStkCZoLcNTjWQQPRVtvPpbInNmBRYqdvAhqZHbYEWdusWOZsBqUXVGEpafFfZUKDRlFSFsfTkAOwpZDoGCjOOjoppvkQFnGvtSKIlHGZmQXnIsYlCCFTfmClhICzMdftDGIKJaGBqkKxhlRSJLiRyciwrCEyFRDjezhIoHcOFUBAMaFVAKfxdXtRTbyDOkxUmyOFLaVldGIuLOCivYcbOIQqSQRFSiAohAcwklxMPIYfozrJqedCfDKUicdRuVrfyQiqkVHXPFAKMStMDNDsieDoBDvLnrYvQwyinIfHbGxZhbgfLbijgVMCaTRERZIdDGiIxWGVSutRvUesRVNBrIxqunDooxgXWMWMtzTmmRPRwBskmlKvewhTEzlpfrhpjTEeCDgjNnpDWFHrhJSCEAaeHnmXiLkuJGenkhmTzwTkHVHcFZrnULrNFfQPQchoLRWTUnqKFpTuvKordsGpRflCOTiliGxDbWCCxGrUCmqVHtTAQwrGFuTjvBGdTLIMgHJlGXmAhgvomLfzojMuEhhtKWnCcmKcGnPnVbmsNhYHMhyfWyceKFPZYrkdbKGACkRzCJPefzmyFmimCGPONgFxeGJOswFcLZlDPZDjIsyBfVsmhWkkMkVDALzfxLurFGhvooGEjTGhHdCryPbkhSEkkQhqNPngtubboGNUDOGHFpQBKhttzrZzekJFgNpJfxMUzFnuMyCNYjajiPfSCZbFMKtKPiPRdPcUiahFcqPeZCpknIuZFeUpVLcHaUtBFMUJRxfoNzgbFRSgommRRjnVkRpaZqrbsJKdedXPqDmjqTyNoSjXfZToXxjzHjnxKyKOYrExTFtdROPQUFyqWtcFaOeBuGzwscyciNYQeZBtdgJUCCIuQydnKmGuWwGXVHwBLECCRrEzPxEVVHRiugujGkaIVSLPQZRyZhlvgWtFKKVLitWThvfpnrbVjHQpMmDDaGkBXhpCyVqXfUEZkRyQlDmsDSimMFrNtkHuKVQVMqAIGlndVCNcdCFknwPPisOTowzslktGfBQRlYrUkEvBwNfhUxlcdoiFDlZoryEdSuUhezfmfrENFkrRHRVElobjfRzanKVmKnmyFpAMssTBhlbTMCCPROfarPYbiivJUkjEidDlKiQrkaZfZpNrPWKYbnkrVKhfMVvPsnnGsItfLiEeZJtxkwGTyqFfRDTMDXDyHDHEgVljiXMoekVdqraXOGHGJtjgVofeTKmXijYUeuXvhPgXnPEUEBBlnjjxuPcZazTLaJhRjiOxNdDtoLwPDgRjfLsmyaWWGYWXccQACHVtyYIPzuXDvwbHxfqvlDErHYOLeLCBQsPbGOEAgobRBTljlbURiXCQKcrHnBZlECjIcbuXJQEJgWTqLwWJAbDGnhzbWrueKaGJwsbMSYRbDgfwyaGyDsenaGifBsxXhTbxZRsLbdoRuWrwwGZYoecbPftQpIMOmCcAXJPXYWCMcYUbByweBMMJEWFuAgArGXaogINRHEwxhwhBOivsbRISgMDRAHTFIEaieVkTXfxuPUHgsBvfahDWNhHhYvHsbXPHqgjeIAXclbrHmYROTiwjscfPJWEOoWNAHQEbvmQeHFRKLurohQkRtGtFeRwjPlrznhROiNTcovqEbARczLNOmFmPoUXCKbrSjDOIvGlLcMvposPssqaYlyDCtAcBDzpzTjQwgoGjhQUQpZEtYVhgZSIjlaSNWgHJkyVNnOuNBNwtvGrvlJxPQnljdZbKejPBygVLswQPmuckPTCujzumxSRSmZNfbLJyUXFKCxCHdcfvvAZLstuNFLNHTahgisjNIWNJFBgGTPNOJxqWVXZvXcqXbJfnLrzPCLachiPIkYtYYsJhwBQVrdmDWiGbPLVtgwTdzoEAALTdPknOVyDuyXYfygAHcAyovgWdMSeQpobcFTvkvUGfBZMkzQXbiOizflZljmWJRwGwVDuHgrRmHHHcwYWdRCVGTAGdZYsCpOvplWVIXzfNzIzWIkLRAoBmFoVbpWBcAGruIYuXbRhOvdxctJQblSHABsCYklAJCVOugUoEyeUPZVLWvFVxotHdAcZwilNIAqOsgFybHwczhEHyaeZBXMHExHrXxXFTYcAgkMZuZiavdDdwcpFvyqxgAuFCezUMyaUzayoPjBFuurhsTkWKFYByuRLgtoiHfTmnKshZJEWPrslKzmqSCySikghfrxJvAgQbNqTJJpGfzWlJKyRlWxCbKHYKutQMRoKhTGzzLjgsCwuKJvgJTLbtOWzTOppEeamXQrtJuXQsEBSqoHuMoaVOfugphVqACLQDVyEjOlhCsgvgvAFmisBObqNvBpaDqjlxDLoJUAYmxlNcKcdSUjAfeDPGurEfdfEmGaiKYGGAXlmEsbjjvAmuPZAgnzgcGCJmoiTFphFlURDnQsbtrSUKDDhWWrEDBOMvEJHpxUvtNBjVabZNdWeRUOUoAWUSrkSmzahyRqDYhXuweASWghekeQFIudhUxgHoQntBllpsljMFQCcycEXhiutETcdbqxdBdVlpfLQMpgagkaBlcNYPwhjWrYahizeZBGfsUBekGYUekgOCuglgIXMFMzrHUHjniRrIGBKScDOsEhdPWFbdMUMYTGfPwpZzhBFIokhQENqrEnuSrNeeoFDzWLGSQKKHMCfpoJUtTRtnXVjsOuPMCbRjRoQUaCeOmshTljPOqeBTbXUrmqHbYLEhOVzgAZUojPZHAMhJdLNUGdVlyhqlVUstzygULJvRWORNUIISMjnrxdTBoEmULqaDSpWchJxMQUNqVVnzdojobhlroMupgLMArkzMWxcuJYpMYLyehjsXtvvbeneXpYHLaLkZdlhwYBLEZFikJjuFENEGskETGNagoOUNmuinirWOfzhUlTajiNFtwvSsgRppksgxLKQRHzpymGWZiZvAUqOLsSAvrZAYebtzAPyeEUrSbkUpAPIcmKnICqpVOeEJcFSbrCTPuwTQBdXlIehkfoBVVhtnnThQZKDqZMCwMdANKjqXpuvzuTeXZOcKtrBtuipIfzuvnxaBFgyQdHRRjgoyMdgUHiuqeraOtThVEgxCsXZQPmuyTBlOrttOXyKNpewbLnjLalhQUaYpsrYYYtfVZznBnCguNxTNMWlQuncgFANcaWvIbAnpJqIzxsCLskzkxzFKnOCDjloQuIXxnfuSYQAUtwtiiCHGWAKYMsvSujMmkzWaVRGyFDfhZmfNTGmGgOiUkJrYYLrqUDSyelkNoKWcbkzfvsjmkgyZYMkpZuOrgmSybGlPbLHDPlokJgcAznnoiFjtBVjeinVpVAzVUisPjXDhLHzGiMpMrwLoCqCLWoGgEWNfZIGSPnDlWmTcvralCICAiZnbagNLsneTYBTPDqslXrIznBUnvCSUcwrzrcxSGdMxiYQuASGqoYrCLTXqSTIgvCJqIgFiEjrHbOvWPLyWpybJNNaXDtiNaSbEkFJLxLgJDzDGzrVmvXYnHnYCWnhWLWvCQWKXRluNYlmiAxxYFMpXcNZimzoqRtkrbINllVLyFUcAoxzemnUtYGBEZcYIzNEasabTnTOlYLnnRfLktQMwpRCejCZiFFhkoXDrYKyrkzJyHAvEKjdGYGTBNCiIbmkcoZZhFuJspNKAuAsZhRPpgVEUqHmSQyjBAyrOPazZUZEtGoqNmhhSzQugjoDmCvBvHpYZebBorPrRsPzJdtYeWuppEQZCOgiQGFrgCqFBItRObryqqCriRJdBHuRpCdgqldaSswMUGfGoVEMIqYvNgLOHXgjOrDgFwCfiHKnkIUtPNUHTWhhIEQFMdJaoFNNHOdTYcgHvvHuYIuqWMLzhgkGOgXLLTPrKQTRKGuYEGjcTmOBjphalIDcUFXnNcwOOUuVqccoeAqTGsbBLVjkQlXHfQQIUvltUdmSzXhzLYILlqEbrsxnouDJGlzLsbpaNKPsCUnXzfJdKKCXTmQSxopsOpBIBFUuLIaDMViXPhcBcvuAQooXHJNRVqnoPoCjZxtCxBUhGERqgzTUZxkWAgtdEkBcHgVVwPShVQcdajcqyTNjEdOhuNDIyzsywpZcHsqDWxdLPreByHMOkUzctzKbRpdHKQuNwTNaHUeyWgYNCKyhHRdqwXfmUSAmVxXKZeEgWHEYVlHNDnHMXbTADmDFBciYcdJTKQfjYXoBYqaYXAIBwzCbqiXiccPVEnnnLpNtOUzMkcPyIiINLyPeyOIIVjxJNaKfTmoGQoaWVZOcgAWoEsbhwsNfhGGxoESmzEsZJcrunEAvwsELVUvwdNzlyeAkyLwbqTwfLMCGoYFhlbiEYBuTtCCrmsxVAIfcFccKScYApMPRYyFTyYNLjlyCjvDaonVeuIpTNmnbBeLzGgIIHKijPxMXNlczTgwhxEaZYWCeSUbTHfedRZEFwMDctKPkcsPsfvlktZCIztqHXmDmhqYOCtrGuylaUflZxNkRyAirgAsRjXSjhKMNMKUlXqpiOJVnTYuknuWKvVyePoKIzQLptOJqhClqPuEHlXWOWhKnhmXGfhVgHDVlBzjxCwRXRXINlXGDaKHqpiYtSGbhFkIIQFLHBcaPVifHYzSFmSyaZCthMQnCoGKMqteEHPUJLFRAKJuiqzOmHlLZgsIWwBFUuZlVIJxmSeOBdYpDoHdTFfacwCmBTeVcDIOWolvNKYzxfsNXWjSQgBwDZuyLBzcOZOkuZpTvAcJQpiXIYvtoICuCsWwWEImJLriTrTKuzVwcQxSRprBJDJRJSJVtjiAufltPuzHAXaahgYDpeXkAdrNuqCPNoqmyCrTViAPlxdVVTNXRYqBxJjWnRNPlsqQaCFNulySQpbSoSdIiDqwsXRUQVTEJhHEuDvpJpCzGwgYBsYhxVwHdlZiGBgfiasaATeIvNGHWbzwwoWHoXmgPijSLdWQgzfTXqTOdePJmhyxoRGkUIPLDgoFemCTyAaXfOlWEyMDHnHHBpxoZDlFMZbrdnYuxaOJEnIjdiSbgJHVYJabYKTngOaTYOmwZdhgybDhKeNIvmcQXzEFKeeNBTIxDgMGqkABQQqgJtuqvgugOytlfsbDEKLFjptPrgJTuGsYKDLynbbzPbnOLOJmQoODtPNbgaEAWVMTRbYqOPTSRwvooFTYPsQjicXASflzkCzfgQTrxiBGtUqewjJDChciooxpkARltPXXfuyUqjiSaWluTiHvoDLTeSBNQHxdAfeXmuwFchchgYNJAVsaunhfRlzTXoIYGnkTMQijoCprFCmfxoCeVzyeYZhNpLhIjeFoYsWvKQTZchRshjwRbmtYGqieREVqZJyBmsrbZALiiaGpZGysYIjKQQRpmqUUlrhLSZANtLdeMgziSCtJhYGTnhcWUYwBLPzQuBPyNcRSWPiHaIobVeraEDKKnvWaldfYmFEnVcnCiVjxucymxgGqGhntjxbZekQyJlJUCQFABKEDiWKVUnVNlnKgCGwmrUhQbVQypZjuYYYNyITRjkZyhZqLlcZDsJmgNBAanGJkhJaiYKaEDsPvSqGMbESFsXRGadxVnVHtBAsaRptKMiIwxHNbgYbKxksECYTvpyjSuAmHhFFYfwdaEreliYfLInylQnsaPeZXpzrMRobCdLCPTRfQcunfoIvZdeOcJvvTwuZxolvRkIrgyRlTCKExTPIbDEzVuQdicHHgaKPOyMchIrwVsFPnzGSsVlUjdtKIbpXoVThagaDzYtGlGWycHFjIDGvjyLlJREEkYgDTHIovswIxuXBfgLvhgFcwfHyrnPDgGjXwgkKCDFgTZAKbrwTXvWKvtIWaOhnEQrPreasGGDQiCbOfviEyDzolFpXQXxiGKKiNiyoNQDSmXIVgwoKEkoFUyZODmrieGAygTxoQvmMhyEqEZHQKuYYvrqlKCgSThhbsbhTmejhSfAjNJtPKhIVxMQkCbVAuIqMiiJMBWNNmpBDaOKNmzESBXkUXDvTKjxGXdXqpdPfBMksdKkJiAFbCICqVOdkwMXFCtbbeqlirGGmVDYvVNzdabtcvHySkiibQwlCgRVsAcMfFYSggDKYuiHsNoBFqSPWAtrjuqslziluxtICrAkFGilfeCjNOdBlagcMXRMqaVawifLZBjdxjVzpeQIqFwAHPEkVCNKCPuABuYwVzwBEWzGPoTcLVeTmBnCInhnRdIXSLftfBXLfHweihzuostnxqvitkZtXEFQjpnflKMatUBPuiWWAZYyUlUmEYISVsaltFxnMHQTCcwEJGxWTgRLRMoItbApqiiJCxPLcRFsiUZOREfBJTWojDsfpJiLHLzodrSPrKFyoekjiPyQnMXTDviapAWwnmfMyEMohCQnsijuQpLrfbimhVaUAoCDEgOcBsBrlPgSZGnerTrXxTBEkRVFNsltJlurZWxTJBcfnYAxjmkBOTDNXdHCvArFnQwLzClpevwOczRphegGtKUAHbdvoMqmYEmYaSlDgrhjJPwsvWAQRJhjEDDZRwSeCaeqQuXNywKHousjWeiFXLrqhvToPTIiySxTBNIqYytwGwfHbBDhIvwZWYzGFkQzePcSQMmXHUuEvZLgiXJTYGIIEpWupKLAheETjzHfJJyClIvZbzMzxIxHEGprhFtoNaBjquwHKufsrbZYPwHzqsDDAdPWPdMOCZbjAAjudDndnDPLKOaPxcKQgerGARxTQyVCEJfHFxmztPaqkdlXJqsHAPmenIiPbZwkAGXgJaEBuhQkiTSdrFJxjamaoIiqdCuyhiZqegACFROOqJPDJgsivXuouTpyFKFkqLjQpHKfSiJElHYwKnqVYVlbVQycmPconXkCLfuNBdlEyWitqaciMBHtaXSPGRdWWIeNeGWECOPVyRWbfxNnhbYHRbEIRibkQgHcxQAHKaynDsItHuDKMevHGbxqmnUZeYsDwLVqOOYqGahrLCgpKkjSJrpzeYTyTdcWHqUBNQoSGRcGRqtaxgTUlQRJkHvjnsGfzsWqsuMoegSXXVxZZugvenXdpdEmwnddRmejYSiagmEbLWgAZrpfKBzvpSumQxYMSmdLfRHsNfAANkxtaRRQQdtqRIVLZEPVWQxgYFVrgJtVPoZzeYyLoLZfscuikGCdPbbtOXztteOEhBsTaeITvoCNAZqnMPkvWZjKNoGruxumETFuHpziMJPeiFDwFEDGROBALjEgyWuSEQDKRZlcMyAgPeSmdabKIFDmXDDiTgLwEMuUzFkNJrIwuQoaAxyWaPOgWaXVoyvgcrorlEnBSnywnriqaTnsILTBSTkakWbMxXfANTYlKFaRRLlmqkDgvKUtEXfMuJprPFQoSxGrUWMIEFvdUWcgWcGiDENAWDfLQukGdeZkOsGHceElzeqpmhBniJrvNjbrAOrdFYUUtENdPndTaiJFmINvQapEnbjzKcpdOzKWuiUPldQOPYuyylPfwAkzxWpDMZoDJJRWOyGfsicBwVMGQgWAhoydHVRMMbCMaSliYsXrZtlKhbQoscVAizfaoAUphgzROjLhqUaxSqWMyjicwxoPfxBSkJTcRLrsPizhMPujoHOmDyNLJeyVjSesJgcnHtgzxRrhZfBkZPVaGgZMJpkgYNvuYkjECxsZlEsdPBEuAKcfXWMxXWHAsqQqfiZdHyFgnwzMievcLSgBJrQcooUSQOOluJqfTZFOiWTugSOrtKdIYLOgXzseEzSHFWxhSSbBwnWXclyYcucUvqVDXKglOCTFyxNSRuONSpciWAWEfjkXHwctvfsoyhyEtJNCUybBsBckeXfFvsxGGzQiUosJYxacWNoUeXAulGySwjHGNwayprfNrGPALVEBlgdyhanQGWkswFxJeOSGcybxFOkJmpXEWQFUpMwvbhcgDmMRlELztNArhmWGMdLBXlqCklbaxPBQCOKVywbZPmgqHYqvUspyBAItVVVHJXygwvrxoGTPqGNVKevSfIzgWoviugXXeMnWshNwjtEgSgzvEDjJOwrDtkBucXKOawkEpjHXuKzsrpgvDpLNEdhoDJOfZYOCeogpQljXuRAxeMgJnTVWopHxGdSKXCLAzpqCwpTPbKaYTBxeIRtGXqyyKiHXrMfUCuFDHKiEtRpTmbRdssiKukNEqglWlBIhWBRXCDjyWqmvvPoKVPOxaUEwZGEpOjxaZknfplntpJxlqrzzZEnGcWBXmJBvBbeJTWcVeJxweuHzFFnbWfFNFaEdeuhyjoYJeBHMfCdIidnkGYAWhGtOnpfYFyTOTLfBszOtezaYCBYJJBkBtOCrjbgRXfafaGNHtiNiFLOtBjRAdBYhhBdKSZshozMqFbczYYZqXvzHQeijuiUDqiERHEBvYYMwcEjhkkvLuZZKybxoKsCWyvItDqCATsQDwtkUiknvfloWdCcrWaaaYSbrwDNyAYQHTDACZWxAfduwOGqnAICsvgTwnmHTzxQjWodBayTtaUZrGMrKEVATUnjXXwjYfgausvqxDkaRpGnggfVIWPgDARykADAolXoqZxCAyZOQADtPHPokXcJvIYPeQLyEcMZWcbYLosVRkKhNqaFOrErAArBRCwwOXosNXhBfkDvZspiQZqiTWWzFQFlAacXZSxVfIYqUvcajOhygNuPOogaojYhakqFrEkgIFiNuvJpUfcyakFHfqwFLyzZsoqgIWVjzhnhMUVKqSNEUvayebpcalKNumvQLbYwTvdeqoSwuqSpYjSexCyDDNDCVHCQIPdBfnxNeoSnjoSQNgUFLRvOYDHwDVWJcKzqJeBWgVSUyqqdQNsNpHnbayIPSvAJJTDELMzaxaZCEOnTIVKmSOHuCvOrJpheATzIgJGmzqgmKWxRvnlomACMHDHVjxXXtiLufFwHpUNHqpHeKVobvxFihUAsazeVCFWExrQuTQhQVXeVBIZYuXMwEqVOHtOHROHnqOsxwEUdMxNNbbhyoQiwznmZbpTgILRfniQCYLqUjilHlbyWklSIdJBHmwlqHvEvOUpNPQApZkRVOXsSdOCvUkLVxLgGGKNwSSeEveUEWIQljRuVpmPDSpfPADFJuLHYuzfSHHWNONCZsQIMLLZtycXsNgXKXAgsNUpzGfmsxaHnOTUOnklHYZYLZdNIgBgaegHUMrvHiypZeLPCaCgAQxtvNxqhbLYsfgJRfQUoVNbLRShTgqKkDImcYkDBlEkDoTGzgqFEOhALStbIxVtFmIamUczLUjeMimffOJQyOSWgfQtMTUscaWEuqDGCKBnbCmlqxFDSGoNXrWRcVQwqCphODlnjYbdSaDIfcqWQnYbccIwLXGyIrcZDIplrgAZUHVedHCLUPwmRTZRHdBRGqtATpBlXPckiBtPrHhxzIniGRORoaVFAOAOBYPpbnLgWOrnNSGdVsQfzecyaQVxhRkVspFAupqVfvqjZCMXMjOdTbRXqmPWqQYDDMayAyfZlqbSkZOTkPENwcApAupcdRGPmlGiLDXwvjdFcNugkpJFHAEFXrJBPBXLrycVgOXMcCnUiJdbmzuBxVTKImCZgIPxdXgYOVpyzrBaQMkArPJTMJTNLuhcHDVRprQOBwcNUeIhSMYKKpxbJYnrKPlYTtRNJGvTQNPBLqYtOnQpBboikkNZdqfcnMKqnAYxsbFiXiAppjzteOmECeEeEWDESHDMoOgcCfwEPIOgmTLjzdVlABtIwxLujWTPsUFlhenVJhSCKtkQIcKFTokcQIJNyeTgDuquUrTmHqIWyOlHIQmecBcgRrnRoNfcqGexfTRwIQFphZokzhqQWAmZaIKiRveOtRflupZminUOPQwPFvjvesBGcutvZfhpqHPxEibMrcKuEUUYGkwKxiTRptsYgkBnrPIKtMLVJSjismfzTIKAwYnxcwOZTbQwGRsZPnNJoBBcADUXqMpVwbAEEfcditZnqxlqWEhFnxEStuWcHIzIXqYwyIlHWbuOoBwoJWzPiPPFVbkWfJvJGiwMcCmkfoqwQISmxBPceQYiqFetvGfFVxpAnfxMfUnZoRTZTiAyFMhWPNCqTfMififdYrZAZdosGZqPharDOALAucPoiKxYPQTWPSZFvyXxPuaQcRpBjxmmtSovpBsVYnENlgLzCfkEPiWrfdkBXJWtskVIOtdsyaIbswjrPpnvFbRQdwkEBoteofaDUMjzBszlgZclovuMbnoqwuGUwGGkhdSvriEHDsUdZOLDqcmSjRNyuUoTwxiXUEQPoJRdySiZlttJGaENudecyJMDWHrckrzRcmolaNMcoDkXreCKsheHReYgZIKojaPVHQlUGwGFEoMwwjvukOSSAUhAQOGvlYVhkafVrKBXXNLooSdUhljrkSoSQiSmcFohRqomEKcEWqXgFYUcPKiRraAZxkruvCbTIBfURBxQJdOkolcTgXMpXKltegslPQGuPUZnfORNpnbOhtyOzMIWVRwptLALDxLspMakjZyLkmkCmsFkMTYjyfvrbOCxzuRwYFlkFkShyVvjGOJHklgBCRlGfhDXlevVslVHfCTrFxLPfzxYYAlgCJxkGLuJmrJBqGzCnfnATEkXqnRQtOUkgPZYtwpjkhVwpWnDnnnhFiKFmfipkVJaYKhvTeLXIqKHNzncJvpCXKrRHNYKmTBktPrRpttHaiVqUnzitNnUCElSKgwhSNFSFbFlTUppRDqhfQrnSmwbLsVlaiWKspfjzUoHhfbAQtgUERwBXpRdhcjFStWEbmFxwWFfzOqtGTETgWWiRgsiemBVHvlkBLtMVjPLaIXeBhUvqZGFgBjjdRxMTUtUwPBPdywnwHAsRCqIexRQkFZLYNjVFHFMebOpETIfCjwwvlEXaXWvXesIcygIWwdjtkHTPkDHAcmPUkhDeGiXGdxtvdlVfnbMaiIqSrfpuSOxRJbnDbndbvPsctMyazQcdCvMyvVvuPhGGfqNauLCQhrMmKExyRXiFuwKGpBLrVrrQfChNZigRUJEqVzfbpINtkGwbdmHgREYprpMUPpFArPhPRYefClrRHImxOzXBxBsHxbnbGKbnSqpmcnnOEOGZMUAIOvVHAhJPUuEaNpvCsAMqUANGtbRTKTEENuyjwzSVOBKecUjgEYkXAoHRSiFqzKWBsGTdAxpEQutwEzQzCYrCULiuaFKWiuIwNYNUnoyQGNNlOzMoPGinKRmTqNMcUipwcrwgMolFIOHiIKdONGxJWojzFrxHFaRbRqDrcxkpsenoqZCQsbaVwjWuZesEFEmtjjXWypXCaeyRcvfNtDdVszsEgzsWXyIXxynPikUilNVkinFpGeLZXCJKfkxTOYaIADTIUwLJMKZwbsBVlGaVIpeETUlRIKVlnSueXwFKJpJbCrDdxmeaJKeXxNKuiySvejXKuBLMOceNUzmvKcXiweyTvxXOYOWiMvKXeonkHROyevrmihyDTKZEdoPvzmbRrOnuwGJxBzhMactsMTpbvqqOIfHLJUCoGkHHXTmFFtYZFlAoTWkLSNKIHUkuGKwQoqFSPhuNlCefNlUrSheKxwkoOVwSzxTWnTOJMSwyFGSCATdxZCeTiHhbhocXZaEyOBlqdXtiUrIADiuoDjPERrtydLPUiiFkZqRlQQMIiwdEJMqcdVDzZTVqEHvbMqojAnpPjuuuMBVjrhGETisqjpCZldQZsOdIaicOSrKZRiCHbUMAsknPksaHOSHrsOYyhWzgXjLJooZAQotKpOiRNxFFQaBvSNkUsNqhBLEkaSqZHcTOfNENRMcdDDVqdnHmGuQCeTjmTglkPWezpkrlxGNBOBbgCbiPkbojpCeovnYIFucZfVyMyYVTHWKeJuEQwZyNCDdqALkDERkAoRSwFkMLAubieeVrKTiTsdLKREWZdFZDhUTsTXRvxMBySyGETjIrOfSWfequoVfGpTWLbyIXkpfDTmsWFCLFjUHlrQBvnFRgeFPhwzqTNwgfBgzHVCpHZfDfaRTGDJxEIcCguVwvevDkqRUTDcpJeEkjSlSQcMQpeDqAAIJPWlwkLfynEVYwXuKRgGruHrJlPGllhBJasGtJULNoMDBpidRSCcxlSMgpHXNYjPJLdRawxCHdBCoKdpQZHAFaSSZdrxlVnwJFCFKpuAdutCysCTPRKqcrbOIMXEivEHUKNaSALpNQYzoFWRZYRIxgXMFqUoIFjbSJvyVUlGan</t>
   </si>
   <si>
     <t>2026-09-02</t>
   </si>
   <si>
-    <t>23:25:32</t>
-  </si>
-  <si>
-    <t>2026-09-02 23:25:37</t>
+    <t>23:42:25</t>
+  </si>
+  <si>
+    <t>2026-09-02 23:42:30</t>
   </si>
   <si>
     <t>{"key":"value5"}</t>
@@ -560,52 +545,49 @@
     <t>&lt;root&gt;&lt;key&gt;value5&lt;/key&gt;&lt;/root&gt;</t>
   </si>
   <si>
-    <t>9223372036854775801</t>
-  </si>
-  <si>
-    <t>Xo</t>
-  </si>
-  <si>
-    <t>hE</t>
-  </si>
-  <si>
-    <t>xu</t>
-  </si>
-  <si>
-    <t>Gt</t>
-  </si>
-  <si>
-    <t>uglSPeSvfxqkKRICgDoFZpALZrUkkzJVbsiDexFHtaoZjluqhtPsdXDmrqqGrOWsPmnGllQQTxLwiCWjgSRmVQeqXmXYutHIRdoGbdkqutTDlRhXSPCnmJbvJwigslfjJjmkjUDAzlzYAvijHCrtDKTXLvmqAyauloLgWYBnBacewwserJeAHmUCogkqYdkaGsOzJqClEGRWFDkhBSkynOodnBRwiD</t>
-  </si>
-  <si>
-    <t>kukOujwuiTXfmhGmeZmGlvgJtCYaPWOPVKgbsiEMHMBdWiFPUIArvcZRSxuSOsDeOUmqrbasDtCwoQtSlTvHTlxhINZxntXarxwLJwrkCOPwAuZlHjQrhqepQacCRLeGw</t>
-  </si>
-  <si>
-    <t>NlNaEMEThHoFQfzwfTiJrqMBPgeMZNlZlXFgjGdaTickINjThhmdmxaUBeSNbxUPwLulUNHuzzjFNiKpKHjIztusPsMDtACkeLOsqBrkGyMGYhxnzlWaLvqVexVLEDBCRbEbUfbMDrmWeTsILxuMzXbPDMzCIXLtvQwJMrLttvkBORtzPPBvuFtSLhAGpDagltmDMcUBWvIFrDiaRsiWGeL</t>
-  </si>
-  <si>
-    <t>YeqmfXiiNtLeLkHLqXOBIBYWZNiYmTEmnlPXBVkMdHlhmUdAMTJnvjsEIbvQuckVPEpjTUutKYkYjEOompHFygQtOmxSmFdYysctpwJzkrBJLHDLfYmPtNtLoWfWrUCbRw</t>
-  </si>
-  <si>
-    <t>JxhMkTqXsEzMkXYDhztIyaFMzPYmNCNhVJrJRIiJLBSZOkYbclUKriATJhoWzaHXNXXXjrwJnTHUYKgsbVZmUjSsgRaDzqEuxsIxhqDKBnDRFOkdkHuHgUKrQcuLGNupKHUxmaumrEfOQfwUgmcSOHgSkimLNMzWYnDQXBTRQCglFrtJKtsJnKjZUYkhYXCcPMRmmEFSnWnSrIKPGxSjulOPcuXBYzkGDKliAkhpmKUWZbJSRmwvcFOMwMuQLQKZZvFRsCaquzNiXFafpVLcxfPhMUgxkIuztMyITNzYuEPxzzrrwthHyiYBjvDDBAvCvqjUQvhbSUFHBaJALJwJpAOsbMyQnDNyagaTjudDHdPLummcTbCUxvhULevXkbzLYXxXLKMKhpmvUBWClqqAKTVomkQsIkHiAiCXKFyUOycPPxmDQfGEOJUpoyqmTdXYOqhGpdFBkqdEwdLviCpoXpJCaiQPLWKPkrIlQCkhiHBaKOXjPWefmDXcHvgEpEZWOdKNzzjOZCcJIfAerkqAjVftPsxZJEIHnZpIIHfChRvwJRefuqXjnIFotTHKddjumKgXkluQkmwYmUKbPjqCRPOUsZastvCqbZNGNyloUSGYZJtjQFBPunjXmiBgdzZWEsgPVSktwhRsFlyIihbelEkaXJvMITzsHTBIKQDVvWQxjgtFLwqisqlFaodXtkWXyMFKESJmYkwUglZvBAYtxnvFLkwRVoUywnmKuhOIWneyVKAcblCtnMQgXgdVBQQygRdWTFxeVLrQShjrZbsKFGpeCYIhhKmXfacOwzGRqIIWyWwhEcAKwyTmqYOaPKRMvQjNKSfrIixQXfXXKVaaAvERbusqdNapgSOBTdyPYXBTITOUNQfIJfUIdKgRGQkzyGiuUSQyXCNAwmtSzWcGgvvxgIyrGlYADnZElCUGtaiPBNNpiZBxInLSpoqCcNOEkRphYOERMWwDEvSScjNXaVixEleQlIPKFukRjUvzLnShaZqduoEbARcygpDLKIgXDaXVvadpmCXWIdXatTAvRZDEbSRzqTVCfpxBYVuGCtYvwrbkWrxHXESMouIclMJyHfCSBSIxFddemWhtAiXIQWacVfIDpXHSzHxcExrSKQyuKKMnBbQqQszNrbxXTJoXNCzjWAooDeJufAYmhzDJkTtEYDscweZuETFwmILaELmWwSylOsSgbxRkxOimiLBmxkmJdgwlbkojrDCldIsllcGGifkIGNCknjiGxRtDjmGXRceIhUsJatoqCKZpvUDcIvOggnMgJSeUcSDwzvLfpWxnTrvCXKRstddICFUNZThFhAjcxYTFSVbIEBfUjvbXNinUzIoBEpfqmUFEfvBAdzBEvgscfnXOlGIZcJvoAWojgAZDsNWiquqbABKKzoPJFVlzZvWmcpGrhGWqDyWRaYFWrjerYGwieAcQBWlNZTyrJScvPSpEGsBjVTehMVgmpPWvHfqUSaIcRyfLFgxMAPucfvjYdMHPUqerCpqYTpagfSRmfpuvHIxgBogpRVCADmVFkyahQCJvQoLQWfQmtzCEVayplgsPzCVJvOZKQmjwvxbKozlqEDiEpyUlabCVMxTTUcdqIunkbAoETMozGtzDZsIFIIAUeaFRaheNTQyUdqoDBKjyIMMziYmFEpiCntMbrHwUdPtFojASnoNHTcuxbyFeeyPMJklDkWDGDuSvhlPchqoGziLmxJAHUPqUDJmtEaFXBnAchhOyfNdvzinzjDRdfwzDwUtVIythmZKFuliuIINeTfyrGybUZiaPGeOxyfhNQhLHJzdbUJjTeOHOcKBBveeUwtwztsUWmDVlgdMSQQWcAVUlsiVhAzqLZQbaAOQHRhUtMBUHVnjgXEdUUXYmRKjNxLvMXKziSecyvdRZcMIKvgBeivdjFogXkEGfeYlfLTjtpXHmkByNzHdgzWACDkwPNdxSivFlmBEHAfPjRGkLHJnOgatBjgVaysLPxEDhKzVhmhiRkOtBtDjpMiHEbQcLNzeVpFEjMVzffSIVtuQABfoOQMFNfDLsfkgizcfPrzNNZRghNBedzXkgixuTgqOxemFSNFrvdUHHVgImhtohfbbnlzZlzLzybeycDLRXTUMrEJdlaHRtdmYxjaHIQtGsbrNsCcQlQerfXqShVDpRqjMyEZuCKPKkpxouUNQgrtrFMvfMtOHPJQfVvjpCPYTfcWaoceatHNLSddNJYWFHJduGPBkNsFzYlyNxRiUqnqiIelaVcWahddFSJAhQkdRZPMMAWWfKfusnFJOoLbNUXZbGeIzpcSzTAtsxbXrPzaVIjiFXYcXolPRRkKcTqbNTOksBsSbJCWyXtbPJEodxkricHDFkokYxtBwuMMnXDAOtCNvbdAsgRTJXXUbXuwtFASpYgyQiUurdbQMiwRxuICfXWaXSgamyrXoMCLqgZcylclsJQleYeSEHfruluktCXFRsXBQwyRLKGNIePRDYbijJNlSmAKqVamqBzvmhRcnSAVtubwFnxqkruDYevjqvEJShzsJfMsgzgFZUkigpSzXxhowraWDrUWdVmFajYNiZLOlZlKWwveXUGZNkOFKoyLriVqjyzgvnWqpiUAUfsmQiAWbHHLwMKyzcUeSoIuiTebozkuOSCewMHCxGzTYANddNMvaayDznAuqBrcaIFyAXBhEWIGRpvAjcTcEmEmjBMhXusPjbAVwjVBpuwiRWHqgqCOvmSeKMgDQOsBngQcEBvUoYyyFIhtDhyXesyuZIDWGGVxozASCYIDPtGvVizExjGZnWHeTgFPUNhAxuanbEdGOEFLdJkNomZAXDtTiLlDbKxhLemjWkcGUsNeDqDcomrHrbzNfgkiSpHFffTHwvORypBxHxaxdGNUgBkgPehNhWjRbammbGZgOtUakEIwlxhRRmjCHgRpOYwFpawyjuyriHpSyAkjERSedZXQqdZGqnGUEZnwgYgSnayNuTJTbIkgDyzNQBxLvFgVpsfgVkwkLhNFzRyTRJiwvTPeBuCMKXYyizBdWgioRUljXJOCshxABFBuBlnWgTgqmLPWDsMuEJTmXnkjcTFXAORGXVtebPrKBJogAIouEOtqcDZNSuZjjfcfvBoYaDHUWxBLIcmqWvVPlipnybneVHygjyyzKybfRrFPwOmtBHznrrEPiZvsgZXwEBBuFaZGeYeUBggxKrxhNPvFQEPXYnnlGghBobcSrxHsqYzwIPJYcDkojwKIRGYLmPqKQaysxeiFfwjcpLfxyxXCKEQzpZouBPfquchufiJcYFOKedXNJJWiocejyjcRZNOSOuugBkbHdxkCidRhYHVwTQMJtGjOefICxfwZLPHVsTliHyesosHhmsAitWbdvVVhblCEIOfiADAVlSmIuJNWvOZCzqmzvzEFPWwtIEjDhETOXKUHkAbqAEyKDEiUXRxbFTLhRcAhMcFZXZKbVBkIHGhTDrITberaLfkZycmEhaGHIzYVvjpvnLJQGdpOZhEaHgqBeOHLIHEyFgbtRkScFJXNvpojXuwakwhqtYCpoDmiCqLSmLHdUrICXbcRLLBFphaBjUMFxWkIihliKeiwzMEHBCHmMiNrDQtirQqPJdeWNujmUILrAKvEzlrswVQiOshJljSNafDsuQfoBRTJkDFykihZZAojmfIRKxLbQPVWFWEWIFAkQnrsfNoRunDxccexMPzWneLVcjKAoDmPlNUopUNoHURMbOWyTsbGfUtMXarYlKDWaYfuBnElOfQmhWukKpsEOSedJqsxSbgMZGWLUHeOKTjLPzRxUaWAIWmNNBFteEulCOZeijNWIVjfzzWcEhbMJPbTYesmYlGIasHRwsHqzDQuhRvVrOXUfBypvrfWTWwDznuPFXwnVWZWWfdxqqqmbsltBCxfYDjJcQEGAplPKaidAOMtmNTHWunlCcnWNCrxlSbMqWwLjstSiSbbQkQwRktElAzANydhpngaUILUMKnifGIGoRQCPerJxoNjdPzXUAgWDOsdmawHUUqFzKdTiyfKNtmNApffePbtahSTFpNHseEaPuvyfFwFDEhyidUIDTyrgiPwQKAVXWgbGuFObRYvpCEchCASbbrhcdusTpcqfJoYMJvpjlaaAbloqDFaDWtIrVCopjMpZPEMeTMowDinVWbfFOdplnvDBDltirdNrOmYoTKvBtclZaMXCFsQCESWDvSMxvbBpaWZZQeihdBCCGUCivKcAbRvtuSTbKGUFPnvPlXruaVcMAjAoEbxXBdiwEmxJAzvyWcyLugnZzXXQUFCqjdoHCGxFUCiXxuJtizxVXaoCIQqIPmpzHrMnulNKmqqcBgKuTBZOUBREuRODrAhdgDzyrFkDXWoeaBiMXQUlWDqidoTygyePNOVlRdEorlxTWFgMTvawcmUcijzajFWlyaCaFGThSuaKevpvrQiXBbvYMPQfEJOgogmrRdUsssronLGXTOjFnMbGZfrdGlVLmaUNlEScvZRYxpRxTTnSPzlFmIVnkHRcHFyHnFyfdzypEbwItJmSMWzScJbnctWYiWhAdhtZxwjnkgUfHOIunZgviYQVmkTzrmlOPYQOrSmnQsmNPxJcKRfZSNRQpYZpyGgenOcZjYOuMgTIvAHzVqLWMVPTPLLERPUzSZzXEJxdPaPQndoeDLJrFjrEBBfQKszNnWrsJfXvVsgqZRDmZDLZTlXfIRgufsgVVxlOLETIuOrItLlzREAMEYWQwKNXFnEYqaUNlgoQmvUTtIWvyeZDnVlsOyocjsEpUvPaiBumBUDdjUqkQNgAJBOoYFNnKqAAhlesJQicfpWivXBbUObAlzZpcTZLaRkqMvLULtxZfJrykKcSGTynxlCFMmswLWhgacJCYjSGQnDxYworhKhuvZFBqeXjmVfrelAatwvoKoksrEWZetVNAJyfULxgeaGttBhZXPtfIQKzEVtTZVZYcBkkpWIsZloijnkRKKLIqxYIxRuvuFFyJjdqfVsmJQyZKNtflZTsvJqqpxYSouYNyaWJorXElrNPvyMzNQQRxVHzhLWQULMMtfdLKXVhdeJjbVzuSXTzyGJTiIGJrbHOUZlDPxwcFnGUCABWUxJVEYQwrYopaGBiBhEYviUNqGYHyjSygFFbPwfXcYjveUnZEeEpMbeXTZOtIVxMcQAQfEZlgBEJbBEPfQrlSSguiIGqLZiaMsZPmSKlBtGfpJlFRPgSAXsSxwOjwugZoFOUfezhrmnKiyewNnbEIZvSzbarokWiZjDjDOtYRUQyQRdYNDyraaJQXbIEtmRYeYxioAIjTsAHZGNSXnAmOAHffYtjCTZjMaKgOYIiXfTINOYByOUylkchibwvHBOKAJcutwnuSGCKoCgJBQLdLxdbbHBNgfiBdPAJaBTCsTYvHhOYgcEALqjZSXWgzTVUwDBbqODwHAXnEccnBxXvTOnwZKimOsuyFajCxFUxBvcqonOBFwwsJDTrWcHlLhTCxoTJIeojADfXfhZsMGqwFhuwCaVWffAlekhwDQEcIYqqEyERtmsexvRpoGMgOwdXhSCifcpMOijNujOJGjdVsEhFaPTsROEqUBjDASklXgyvgTdvKGOFMEaCDJHuNNUodzTwYOwlZDkHgRYTgHSGWRuaNQEuVKnTawCWNMYpDudcznKvWNZzbiHdeGIcxZxDfrjLymAnOcECSRGTBigmhqFeOWyFAHneIqiXHPtYUsBAMDtcaHWFjEIrydDYTrznqnIYXbFfKkUKytCNNZRaFQwwJQEVeEvsErwLKnoZkFjFqDOOIyxLOvwGysIfdwBzESWRofYIDRbkjkQvcxabFXVEyLWtSaXpWVyPCKdcDhaFvLdfNArRcoLekpmmkHdjFWzkdmTlWSzYFoGFNqxatdiczsVUyHThlwfEugAFgNxySSsYxvIeSncnCyspjwkqfYZAKYPplQSRzBVQEDLmMNyWdbBhNMoutqUJOJyilpqrngVusiTvdtiOJaPPouDNRsGCqhLVtWPDeJCsvNdxSaVDiNzHUGjLXbxyaWNQwnpgPiCpPtEKbGyeLUhwnvdMsQbewoYaVAKaLNkeDsowStGNClXyrvhqRzqLfFSrHQpJjDDOIBAQIeSJVXzgyoOUXKxuDesaXkUynpFuILEaLhfCYBjgtGBvioMnaXtarigSachmPwPlQWFgXfSkKNvqBUriSvLGhlqbtKPpoNhYTkAtvbGKoswJBuMbVlfotiQAZvleMHAMgLZLjAndQkWiYHBUPLQipJhaAGkoeNijoUpKEgbnVHeaUorKUOrHAGRfjUFAnLtoXzTFgzTfFOhHWyxJTEdkCRAwQSZYlSgLCwPspkcjOMOgijgbDmVzMAKEsPBtmAcKkzXgGcgUaHwZZRfqOmBMmlkMNFoamQEIWWFllXdPYEfowYCFwwLjlRrEiqygLTBsHVibzEOrvezLFYlYdgDycxnlVOURBAgnHQeKmXRKpxmflUCfJneHXqlCVDiaUBAjEjPqtkAgzlmZxkCxfiSfjRUblneDmxjnkHtaZdsuSnZhoLQGgylDYbOTqVFHCMBgXwsnXGpqLaamebUAgFsntCmUjVNNSimFAvuHQrABtxdbkJDNDFhfMMxhScIEPLMubJDKIYNGhuDVJAOssvqrYQrtUBpcHaxIKUThdLlnIMFlmQZypDaTLxMVaHJwGTRKyHdFjYUViUPqexxuUBEhgDATDWdnTrxmVVtpuAQIDqphPYIleTrpNOhOjAMxHdnlOkWseocKRoOMTwADQCACATizLKPlyXpZinoMHAqQvALBhsGOLireTumMswnWKQudUjonlOcJEZoErykNexZLSsBiTeYsSkvVCiqlveKtRCLJwQuPhitNTMsTOrOjgclFerwdMCWdueEnPCaOojUuHppadqXNcVvAVyzkpevZmGZAsHnYfpUoSHAmowVjEaKeWISiOUtRluInYuWmUkqzAHmcTjcgxUDbqxGuTpzxNMUTKKZKqKpioFeImVBUSPGCoioSXZWUCrjwyPzLAoyorPskrXiWgWEWNeSYymhevKCIMNLDCIOGsPnKauRmoknewTDpLcaCABVVuDSBHQnToabmLHkzSqOnJyJRGoIxqnsxoHbvgbgKwuOkRToTFDFfMoCmaJRjoXLmKBePOhQcNOtSaiSNjYtXZrSvpmLYPMFMTQJgmKovRXzswzfiECyXmiCMcolgCSvVIUqqISZxXWiAKFOoTdoWJzwqTkNXubYjKMVDDbixVqtdxkmVExdFixlcTULJPnfQAIFbHJahjYkDVUjjHReQWJblSVAEZuoddmmWwSMhulyoaPiLbcLyNjliPsDVoieCJxnLvqYZeLsbSvJHEDCURqOsPTvLKJoWeateuuSfpGRFRbNxjkTxQkDryyNKbzmXNdBqDvRdJWacUqdSccAyhjtWMnodHERHoCaHFsWKjZVNttsFmiYbArfCwnFcltYLADjEHghAZfIIasACLhoNjMeLxTrtBqGVcwmqSTyBmQfLUApreOuqiRkZYoZbmiAjcOogednANjUlgthOmpMESuhTucJXjJmUcUuVLWCCbtQRBYsPRIubKqHrytvRuVhUNADytpzAxixXYTQHPgpNEiVNcImDmHvAnybWNTbCOAlyUTYBcfztezWDrsfNHHvhbhKqsKDnQYOWHgPyqrdYqdkoxlEGkVXwkngrnHBGTQpmsTUYFgKkZUihyGGverMWovEYycmosSruNCiuwQMMnmEnypblZvglgwQaaczXtulSoOYVyaJahAQdwXuDHqFoSOCXMhkCNkYanfeRxfMhZDkrWeKgoAKqxMlYDwMJrMwUEUCvBencAKRgcSNUAUNZFaTVItHKmdSkbPjCOIpJGYcsqsmXzjHdBurQipFCZdRtaKLplppYsfbYrVhasJEfXMEshiJTnIYFIzLnEokPbniEepCfWulGcTgsGzjkFWJfsVzmOBmtIgDgCtSWPnmvSUbJTIDevBYVHHzIyjBlSzCXRemXfkzIyofQXuYEksHPWzxgElFXSVNVskBHgQIRMgKwOltBilJMpBCytrSfHNWuMTDVLItZfoXDelNWhKIxyDgBONCpwGXZmlBOCTRDTboTZOMXRxdSgPBXJtIZXPpOXmhnFmWhXPTwMuBQNqeDMwpEvWXTxogeVvTakHmSGhZaGlKTCgjkBMGnKDVeMxZsEQgQQaMZYaBbihXRyMqZVIQIUMDOVcjXitWLvovyaoMRvWAEMMLRtusglooMosDfTOLOQCuhMsVAvNTOGqMZfhVGHhPOQAtTlOXMyTxsxVVzKHEBkqPBGfzJlvjCBpLTeVqMHTOobJXXEQilwSlVwdnExXvxFvnTdXjIdBllWUWTrkgNuwoYTojsNheMKZiEJaJROaLnfyyxsJlITssKxtokCABUSprZYVZPIvViEqljxGUZzJEAtcXNAUJHBrEpgabHZPXyxVFNYQsDuhTzBhOfxBqSTBkoJIDUkfiRIwQJFiBdHnURKaLEIaLuJdCXJEpmmudwkwjtjLVPhxJvkUCjTljqfYxYDFfuBGsNXEyaPdFYyMFrfQqhDcPxLYDszCVlBGwdOTFlpHnShufBNFYSmILgsVdCPIDNLURRADoFmGrYVHsbbIBQpdlPuGpIaPUcQiuHmbRRVwxggFvYhXyhJZvkyblgjnHjCyWPdPdbgICalUIUfvAcDSZucLDXeJFyxwjadmpgJkXkWPWXxJKTpenxJgOYNTTcghdRzzhRfENnfhMoQByREVuTNRGyNaOGZOjEdrMWsGpTXzSplvxtNEkYvmXgJEUxfKJonWYWzFZwvArAfkXvrdWrlqtjJvZXMQMOvbwQcCWUBAnamxzvCTaJseBMecsHyOHsLAHrDdHJFpaYcRhOjngADFjMHdBjBJJkaJoyuNaFJgmdZhJLlRQLtZPvxZTxLffmrprTEPVHzKCzutXNwGhGlJfXwyEEoghfLrhOJEiYdnjNXQUJJTHHHlZwGZTJQdUGLuaJuCGAayEDuPUXOmCdWkAYrPJSeCSazRrtGAfukaMAhibmovHHGTukBbXdlPssitjRnRjVdslUGKgDXuMRqJCZPLPuVAWMjdycDppLPwRFKXhMRBgqUSEiTCrJYmDOHNmVRSjJXYvEGrGkuHkyEODTtMInLrNtFfzXdPbgUBSOorkQXzyLqmWhxFPqDayBHwsHpwlVFGZLWglFwfcAhZHiPyCQSHJgNSsYowxOcKmxsFetulfiRmKscDTGgKcyHJxSqdmtCPGEMCbIYmMWwuFYkrKhvPItclRDvJWPhkfwMvTHWuwhpoeANFVUxDOsxPwrdoVETfOzXoaMVqyyDdlPjxZQqqBXzphDggDiqkJGXWuXnAtcHMruwOJTPtRkEuqLhfxQLOkbnXQXJGoIRnRifNPfIGKWMwCcUvRFFdtqSwrocPBWbEApIqDsXijICyocqrWvMegSqxbTyTBkcKMrqfXjOXjkpSJJfjDXEWkjHQzaVsaBtxDloekvdRimFQbfEncrpRvOtkgVBQAjrYQgTKkjYpsRSeCubcEOTKtLzWbDsmfXXOrLVegrvXGWMKfqKltfyiHbPoCBJFQdilgttaUTqEPOrOhWkgnPpfjrKwFPZzBGdoyNZtTmnxRzAyYHvuwfhfMmZYGvDVXCOuiIzGZuQqctRbqmTKmoVsPkZUyUggtqwCVTibxuXflndJkojbjeFZggwXfQgzWLBUuVpPsCEXFTFpiPzHWJCmjBIXhEkPUimvisYwfsFQPutncyJmaJCzQSpXAHirRLAAULMaAhjjhNOmvODuxQFlVoWjCgzRsrsCaWlnHoNRbykEFtRrBMxcxgwQmHqDmStvpVvfHHgYFjWqvKqtfaZTrqRFKlGjXldABQgkHSaULbrMLSEyQVhgFUTfTlTebMbDXQpquAoiQpvwRGhLuFQsdyAOiPDiXctDUEkTgEzNfvFmhHuURRKacFtrSPhQnsDpTYQZZnlceiQqrBbxvIBGkPQtduCzNvTDeOTHnoOLEBOtzUjhDjqqQLOhNwuhdEJVPFrJFiZmQHrmdxENvpMRKgHlVUgWZmrjeUhVTymQySBxmYuxvRavazCiaVxrhQRTHHbRnWfNVcwnNiKcieTfgUJFECKOhaNwRDJDqNxyjXCexOmTUPIGTAnetvDwPeGalGozigSKrwcFhTuzCDHkFRUSaDflUQmdJLcjdavxSVDHKvjSYiwiZNbHtLqVMvMeZDxoOHTkNCCmVIcefPBYnDjNlzWovAITPQumUzrlVVjSvxmZFZccSoTiPYwKbnikwzMVHHURutvxkGIrhxPxqIRwRblGNSgQxvymrsuCpAmVNyRsUyCQpLMatAtTWYQxXXLWSMEuHbteNiKefOwsBGHuisBOfxngcfOzZJkLPlqPnEjINctXhllgkkarLNVTadiWmMvWIYXEnOziPRMBCVEbUUzylVFPXQsttUBOLvvGyIPIbdgshrAEKYHybkxtgUEiaSjtqxheCiuZPGjjnpwBIFPSaVlyxmYLJuwSUkRAgndkTbgSDBLnKKNsfncdSNLPGFeWWauWEfXioNqwTPoPczGmatWCyRThwDPXUGXilXVHWegSkrJiJghDRfGtIBbMBbzTWDJIzSWeHOEsCIWIFOhTzAPrnVrplXfznDFUqTPyabgvsdFLYiMyNHRwsFhBkxGfNSQWFAmXnNSnRQVOrivKsPKHNsdQvxGBroUgNfVigwbmEwNxjFHJeixJhEXKNYIGbIyohCMaRwngIEzFJtQBRKVwHuGJZqqrpJbsfGhPKINhEoPuQPbduyuXyddepSZgKrdIfKjUKgplTujfpCUAvMkgcgsTaECISTPiLGnqgIRFJgNJrQipsfTGzxQSnuPiFNvpDiByImTHQMllMBAxnMCjDgdmwpuMuVOUOmrxdAnQKdTeVhbjzomJehPnABSyvMpAdExceWHsgFbGZUkfercbRvUPjOZhNjfrORiuFRINbGHNuaViNQWRbMKrEqOaeMwtcnkjJnDcIxAotLQqLhaVDiRZUNPOcEJXwniyKolUSvewxrkjsGYaZdxyUnbMFZvaylBpchsRJdAwweRfmPssiPEMHboaMFKlBVVNxpMBvrpMfKokJojERsJBHpeSkaDcWhXBsQhZOxTEBvlQCILBlZNHuPMAwYAacVaBMORpCwxLnhRaIOnHFImTWGcoWmjcJfUQtdfnbciaWZECraivSqIBlMkPYQDtHcNsJVskWYWpLZWpXvmJhbgyEnEyGJhaBowyItraqJuGrXSZUjPsfLiamHfBkvGkxhNdacnolnKsPweLrsItvAmEMplKzfjHoITWKyHetRWphWThTZalphIAgJDihethbfmCVZfNheYRCZoOZBkevYWZMylUiXZgMckiNOJOxtLDeXayGpoFCQVGgBwREXNzciNVSQBGbScbEWZVOqFDvrtLhSTdfzEmeMJYaYIcsZUhPIyLQmxqCpHxXPjsaIKDtrMdQhqjIfeaiFWxHbzgdIZVAEZSQhJIwyWxNEkzXWkHpYBgWXEcttYhqAHmRzAbiRxclFWtnMcKGGfWDdtzdXooNLHHysAZsRCPivsZbKElyccBQRXSVizAIYvfmIjIqKVCCiDiUWfShFtmBRBjEVEyoivnNlZYrHTgOXJJUApLRbFlYsyWwfUJcSMqcYsiHdyZdlZcxmFtBUrgfGHzdCbcCUQbJImTgRttqedGIVvgBqCGaaNYgiixHTjxsRgTtvvntkiKLLBUpvvzFNcnKYONjmwhJqGxvAzufscjgDYfUVeHntMtsyiqSVBKhblPANkWrGEjrnbYukyFTeZVmWukaFxzKKFYlUNhIwszoVMqjOnLrovBNmWZudScHyIhcMdwFCMZWlpqPQfFZlFVbGQywrbqairQUpFpRPsbBNGPHLursNkuXHvxxwQJbEPPISuPqpoHWllzMCBmoXXNhndkwYpdWUIBheAwgJXEJIiSDvUPmyBfnQDRSQtyDtdWLlZmmUOCxQvimbCuAIvQFYnDPwJyZhLmDGAetWKiLBtfgtJrOQUHqDJVVdeMcXWWLtUxVOfulGjeUeQrZurBlxAToCncvrQdPHfcloVEgNnTnxoSXnxNanUskbslVqwiOEIdrSxcDfcWYESieCoUTUQOVYKcevvKFudkhLeNzQtvtgzUAsClKKcCimnjTYwiKDOxYpaLMciXXiuTxPkCtVjJcfcvqNwLXsWaIddIhVtvgpAtnTTopzmPdXKTZWomlnefAwNNxizYNQlFADXPZqJVeyXPRJovBbmMxRoVWPGbguymkGjClbsiyStvIVeKserMzoFPcArxPamocyJyqRrtUsrQGxMqyUsAzZwUIWyXCNxmXBZTsqUELzuVJMlPVERQHIKdcjAmLvHLhnFwFnrFcJBbmAXDCahYrPcLmDWeBgtpWQiYaMIPEeiXrNHIROccYOvqMVLMTCRQJypNGetreiRZtVGRjwUyOuUSseiKaUpXZiFgBEuugqvRcOWTGzyyaLUcGkzWKcoJwGtrBZjUZcvOjrBrUmgPWLXPbVypdBKSpfSaWqOKqsyCPrpKDIzCuSPQOsIsDkOdBytJCklWZePOlJVvpPYxMxRaOSewCuJZuluuPtQsIycdgxWtXWJwxwXbbuSChykGouqQyiKSjNmxSJjnbIckNbwUdTPVLrNIPqAduVuzTjzrFyergEHwdguTiZpmhLHMtJRXsNETJVQGEexrlcmwlhDPQblypoyeTXTSOYLqzUpusreYCVvDCNwBFXZViBycNDcBYLaNnIWqQPhVrEhKGHzjsNsxtQhJUwjDayVVnpQJfnPKSzHXIHNxSQDDLdyHPeOIcNaJrzYKaspaGeprdkQEHQYPfUbmXnSKlVfcygOYBUzDlFlAkKnjhWacAOpRYjOCGNxYjYoMTmCftUvLRCIXpierHZDLmVQGyHjmESNZLBJKRnPAHpWATfPgZiuLWniDHIzYSXpnSTjZjmsVRhkEYadSVnBNCBVhjopuAKkovcdZeFyAszJsdsEPuqFnmnIqEwzOAhDfWBzhmoAQofKeCUVZxVRDlCCDDeImnpEoamBpbhOsmFirkXDxLnIntuQMuKIfUdWkyRfAghPrYCJsDwoueUyBwvtnitlKINYKPhqQSVSUnHvYPBBeLJWauoNOAwopVXbPwMcHazTbSYEodGaQIcfFpteOdgVvyfGhyCSlWFIOkAUCBrixTajKXtHBgtlDwxhWuaUCxWUkkKoXgoPSytlhOZzDdazTStqoJjoLjsLVjCuUEqBPGdeYRpjaMFpjKNrgicRMUKFrWTKuPPZubYuTODmDyqyLXVBnuWcfobBeDBMbPOcdHtABIAKojGDOVucUTqvbFnwHIRcUqnNIPkSKbdlnFOnfXMPNFtKYZVkktqFpwghqPEtnDuUcNmhIyUGSviGNVxAbaRyzAhlhcWqXCauEduVgBHrrXglRrWiHGRUImWwamJNWFNrugfPcfrpvtCVoMTCAASzkSoTtNssMENgagYpSFsOvLNseJkqupSwHaKmiyIfDthdQubYqXxWBqwhrfNGlkfXUSEjjqdlCihtYxjjNeECnmvIeSzfjLxyKCNAqaMPMeOqJPFFlHMlGMSHtlqGKxsPOXoDdkqSlWYADmaukOmHgbkIZHUtXiwFHYCojSEdgpEXtxtwCzyKdslqDVatrwCIaDNaFvTMoaKnSSBEyKgCRikdUFePXjggRqlTinXWHBffSQgZHeyaHtYORhijkrcWvlGKvoItBhRdykqpVWwmBIoxjIjQdXCmwbINQKVviyGOljuedMPFNsKqbNtPKlIByqNixZxUolrcTktyATbCHjkEpdrhrRgXerObwGlvhzYtPJGzkLicIXgPWiyHjlhJZGywmqsfDcWrPgSdJACmSJWWtyYOeurTDzpznePSlnDqwNSmPPNmLcPJbRaEDlJFwVccHhJBkpZdgDFhelUmvvcnLMPURiHhGNeFCmyxVpqGHEiVJGrKRUtHLABZwRmWZwXexFNHaatlPocZvKSzcQubFhmJelXxWHIXXfIkebPnnkAaFQIklaLJLWLAiAWSYkAveAouvwCrAoxHdcaUlouXEBOcPdTDDpCYBnsFDpRBGTuBgwKgjUQENTdSOwoZxSVysUnPOmEuOYcdwAnUUNPsQowrAHWWpWIODQqqXTbScCapPKxNwnGMZTSeqBsVdRHvbmDGFxMWCZlUtKyyWsWpZsjmbYxHzYFjQpsvXLQCdcQsYVEwZVlwYjcEOgWSwGTTwxDxEtTCwtArhdHWRuyaWniDDNstuuPInEIdOzfrgXxCXTwtugRFKKQBqFnnoCVBaqkwiuQHvXOksNKsmsUWtooXDHqbkvbtBxfHrCbyIXVqKYPQgEJYLoklmTnlHhzAMraWqocJNQGocksgalPJDNRBGIZaKqPaUdvFLdyXqjVbINfOqIkwKqSfCViQoSFVRWISSGjVMaCZvTAmGuCCSusdzLqUoqXujpobjUWdmncrqYETGPPdPUJWlEWjacwJecswUotczSmYnXDEYfbdaixzzRreoAuxYyXxZNikqFhZeSoYttJXztesNLCXyuvrDoCesbjnDoxEnlYXICTXlvLpMJQpTmGIxLLZbrDRsquTUesAgoqZmRXdUPwsEYkjjFlzVymHmLtGkZmONOxGRVVnFyusJahouIgOoAveShmUsYEDuWtmeJVvMhTzMKxzDZfOeCsaVGTtoLHGOFVVjVhDiHNUdkPpxykkOxsuFrQCInRhrrMhDJewuyMawoDGqBUyGbynymZjAJjoFnrWsdCCrNifDMznBkutpZXADYaxLbKtmbOBTgdmhYOHapOdusBLADeLZwjGSWudvQCJIfRZoeaVzhrwrdgLsGGMjQIIDhaiPIAkwOuDjNpjgmTxKRRiQfzZAOHKztNQWVKrMqLPxtilFZXIGpiodqxPFvmQndSUaWmbrFmxETXznemdUyfWLjvwtRKuCZABMMfwFpcQGSoLiavWKRsyLdhRLFtvuCHZVYgPSttNknRAMvJRyZAkBfRgVnabyVAcrbGDkumirDKYosarGnyabpOpwhlhYrnOEMSNdKEbmiYfpRsViVHDEUowcHNgobSGisYktaAJFJJeLswLMLZjObjLWYFFprpJOtSRQEtoHKoKMjayGfWlqBlsZfmEAXoWEsIGeGQXFeiTtHaavLvqEssqfVDrOMtSySkHhvEvGWHkjlVpVTfdIFliHHHJnLIPcOiwroTgaWleJngtHHelcQWPOQLfUepifiHVkhUlMNuySqMLknHYOVtCvvYRXuwEnCWRvKdBtHsKELqGPaSZHRpEkuZOmyzLkhEgeQtUDdYzwApHFpugBUYVnXoKmazqdYFuMcaYVMuVJXumyYRuqZPXDResWhErSmbOMeeulbpAqBSQnZZeHGOQJoBasPzsBCTxQyylZqUhrffhSOUXlrQmsYpLtrsRiIWUnudfgKcxxcxOlXBmRIEQqzVUBQqYOZuBiMFyzcOlAiwnmnbKQYxMhNCQaOrMCBmFCqyKLpOWikUBTTauxAOSxCyWKYfONWiFgnwZcsEWPTNXHUaExjfKYXEIGFzwAZDHFIXxZLaiIyumQcuKTnLRpWbUeVTgztBGZtOALAApoOjXwluxWWZONLqAbblbwRqqjoqHtTElTuhRDfwUaspZicgGfSzTofgFNCJhoQzRtGYGUYLJZVNTMuZbazGRQxIBhfyaStakjmQQDSPRajGBEyCGySMFiwCIDYdDWxTzXQQPBPQyZEUnCuhNhCjgzZekFfxiIcxnbEfmpHLFYeAQfqmSPHTQyvCyKHKXKEvNbQmlAdAkiuVueCzaVXTMQSGvCSKKMyhOdeaLgCwKQEkcbOtabRtjZzoxRXGYdEfJBcpcoRyGokfknSwjSzHDKzJKAFgHmXhblDVvdSlKuukbNxPHGyrVuxwlqPgehjbtWWeoitNLZELuniUnPVbsHJFpYUQwLFYRZOYrRQnMPyFcJvUbhgXFRHhqiEWKfwkqYMeFDGxhOiavQLYDXBwLkyPNUpimNVVwnvYTYjLtvcCbbGRUnzPDreKeooPhpiwJjkEispLrjuyziLNXVwGaDTWUiBnPOiAhjRYfDhzHghdoLjsABMADfSLlMQdodMYWySlPUKweUTQDjkydPhSOeoBCpBfJXUqchmuabUHAFvnCsrYjkPFplQCeUFQYwJVqpdwqJXehuruICUyKDVvipvSfwfuoghHwBANqetslGuycMvdxgEzdMeJDCmqZfwFdqeKcaahORGgFuplhVynuVlzugEAszqouBxeTEuXSNCEQZUSpbdZCPrCboSUYhEjrPOHDQfADRdtkyYIGJvSbrGDoDPreuUzvdKTJzZKaUxFALMBnlwtnqltUamuWqLzUzbWLnTxHhqsieeChoQooaRREwgNMJJeBqSXgieiJlJqBTWtkZZHkIDGZAfwQYdMuhrxMbcfCWwFGbeeLxBOUnZKizBXTcGQGKhstpdJeOCxblalFCmaTWKHxaCsKSRKyVhGtpWdZPYHIjLATiVnfGAniydtPueVkRfslWHghIyssNWaBVwgOpWnKOkPppOpWoKmhTngtyixAohjLYQytVDcigxytzjPYxbLAozROdkVsiIOhgVdETjzKKtRzPCLuRAQYuynPzrGKEZWPhxsTnekqRXSkfdMhIDdgSaAfHdsobnVmXAeSzUOUpTfxTtquPQbeSxPygRZRuexdKwynBrEGunjhsyijiTtjtOeetKyWLMmQomWyFdatevxdDRLfxdQmKzkbbHadQkmYjXQuCOXoaokjnbpxBsZGyjhSFeoiZHVRnHmaGWAHancpaKVELyxvlczxazFTVcRNHiMSAHLNPfRKlsQxRKRfWxAqwSatrxvtmQyvMnCeLuDIotYaoRXFzMKSWxolxzeyYyRUUZIhoZqlXRxUYDRoXyquMeXEqdScYRQXIqpTnPndXzdArznxzxulDvuItvkFPyKbdhRElqmHAGXgqydKTJmvDNbyVkGVQLMIJRGZsRVojrVSHiuZfsEfiLUHBiAjHlZsfFrSoqyetbcexvYkvwbyTiWhyRbPYmYMymGsVOZWNOizALxVQajATvpTXzoAtrDEiNFZaZCIaYGSRPhMuVaqSerRVXOcQvnecpEnYpRrVfIWbeFJBIfjTVOYuJqdohdNLSuWSyzywpZTIEtIBdIJLBmARmROKHBqBwMkvzIvIHCTHigiwoRtrIAOYhYTFIiweDuZHUEwJsNpOhZpiELXOrLcSSTgjYlhYgpBTZPLzKavMJYXneLCcwnbxrUaNhMOhBflxZGJeSaiQVgDMbfLBIzKCBqCpVwiiZNhycUIsCLezKyuxOTAkvkupnFemVqmYTtZCIwFOWAOCslfCWkmzJZFPkjINPzeEjhDkEfubivpzmCOFiOCyGEjRkTRYkWwglZrtOAAOONQKjhFUmODfSarwZMQfVtSGNYfxBHmFmwGguIkPPAwBOXBjgQIvquyAYLfjNCRlDbpvneufiIjzwhSSRiYMdbvxsJQMnKjYOQoDJBzCUOFiuEjHrBrnSuxYRSKrVCUYtMjRiPvtSwZsrYHYuQZqUvasIprBdpKrYnVJZECbiCObVgBxMXsgEIkxFKgkRrwaEmiQUrAZcbuOPhMBizrlYUbFhLqPVIQYNsqwAEfEowZlKkAIJETCRvjRRwQFHNhwLWCrXPhgvtbNWQSUyuKPHTOQohYgzGApHepnUVfBxddbJNCerGecgZtTCrIlMxiPaSPpcbnkhFizDLrNHUtjXPpLkfmzSsXpbTrjuyaPojRmzVCGhWykbKwrQcvACvVbtiQbPolDpEEloVgLHBzdbrMxLkOgKntbsQvMJwFIInKqPQTFOtznJkEsowoRdlgpcQINOsbdVWkUisZlFhqzhRJbPAFpmBanYHZUnqigmeMWeYztORGdIfmZmIhpeRXdUCoArFcgGiluKzrRQHbzsgLlJQSQPjYDETkbZoeraGBMULvOPFoooExEyVacjiggAUzJgYfxuzsbUOEOvJLAZGEdGqcLFXfIUKQQkucGWLESTmsNwbBTcPfXgtASLGUINQpWPpKoCWRJihemknLkPjdBLfwovorVYgOmhIPIdTGUhexgSJlBzASfbtUwnyWRazFrvVfhDozPlElbfjOHRNoGgIyavKxlvLcaeLoiUTvnpXbBQsZkMNEuDfAQExLUvXMemOeWBNCKSSsBzKUrsndkrsDPaFKpbpmZFhVzmmSKdFLONAElIwOkATHthOhfEAVoSxpTUwRTSXFybcnRJjnosCxAktggnEmIODdqIJzCdStjlKMTfebhyhAmgcXtnNVHZVxPSKnwUbHqkfesFqCXcACopOrHJnWjlTxdaKpIWqysjRnGcgAykeDBzQYbDfqrfqWImtbfOpiIvnaHNtPEHwriLfYBDDzMWupWjzdAfnGEerrUQZRrIFqBzHWcXjyVxzxDnZWewGYllVCYnxCeUWPKjfiDRSMhzppgLmXSkPkwLwUURoKRZfXNJFoirqpVSQFnssklrMInRJlmKTkPGjjvFlHxglFUcOTaqoajUBShYBULEYowIHztWkQPLXSTodZarcMKHqXTTriLuOmNcAiyRbnsYGojdHuZrroCHPbkwOZsbOopYHJYiCugfEvtPZsnIQLiWtyXpkEyrviExITRlaRoIoYQdcefiCIGxSJRQmZCjbUxYWRauPcSDFpgJUGmrkjKilZBRCSwEKDNWVzzyXFpBgNRIzkBgaosGnFghblOkUdxLYEOsOhLkPOfFUWdVckBIQajILQSLTlvnwUbsQcsvixVnlOnijqhXoRTKOThmzYakhaorbksfxJtEEVFQIIWEvfCZVTIucILVYnTWtZAqsyBHOXOCryfbXkkIXaFuczLPEXeTSvbSifohNWXEebZJQFRIHWlhtUlyctNfeSbEtxoofLhGaZpePhARQETxrdcGbBGbNqHgRmgsexIDGhdQBcgVVSJVrmorMigckXBbfFXdmUGFBOOubJZMxaxaUxvAGYzOarMKtIxlQWspBtULTtLcYiitlhudWkanfBfVuLlGpCVYsRMcZMvgorYONYqAbVreqypNGplmmSGAmUemkcwFLbZwjybOClskJhGPPVXexPcMlTeWTRBJMxRZgpYkNevlRBJxUAPDprUmbSxSKTVDTebhGNAypnaPWLeuTwHyWtLAfKavgPqKjgPNIbQAzqqoPGlFUQEarpAhxerVKjabQPbuGHwXHuRzUVmmPULgZTFngbNpvGxgucoNywwapWcCYHiTqpkafveOZiiDHhjAMpuJVDtRiBQePiurnerdnpYWqyQgNPXrGYBHHLPzDCvmsiTozWMmDcpffkBFyoRPgvgRkYfsFQavgDLEadnDVauBaOQXvPiTqkOcRCAzkhYPfGlLWKDlicFBtgtzqfdWmDOTvjmeMoENSsrfOYNrxBpLTtejIQzUZApWzYiLMyAZAFcaMMLfelgBrgUHmpGYdHUQjKTzBDObNPEzUDcfzoCVnzeuymHhfEvTJuxGFQiaFvadYyLlYLuBjiFQGOCJxSafSUFeAnKdUyBhxfwTeiIUCBUvSgBaKuyjnKdqmrvLKpAtILYAemRymAohfNgyXrHrPUCtnVcxNWiOJDDBFMjIwQVkgsxDjFVhhynHepDYBuwtOgctMLjFONFpYwaIJSybuXUJaxEiYPFCieEETzGUIxSePHzMuAgSClxxtLtPHEZGaORQNoIGLRMINbSXmefObiwsUFGbwLYcoxZMkpcILrlfcAheUYfYmmVkWrbgxHEDrxsMUaAdqxfgzxTrAAkLIfumezuBefkbkRCTCeKNWRTfMmSDSkLXhjBFYBzwAkVaacqklSXZQVqGHHIEZYbIqbBIdBbIkBFOFrQYGiEDUVDmLjoPblXEJwfevZTKIkmJdXUCkxqiIcGZyYWWNkDzoNBzTDkFFCnqNmXgsSFhAEmgNUEligkckcwOGCwBqwWBoGzkfkugJuYooFmGiWrTzbKwNtFVIExwivQJiAlbDTIFhuzpMIIaAQtREOhDpxQgkphxapFFdzvdAXExKuymVTuuUiozqLjvoICoCIGpIENRgwPUldRrRlTNxAmWjmcYbgpOxiEfqanhEerlcAnhTbaexWQRXtnZFVLSgOBOqbLJTxLtjxpNJMDMiLzenhfjlXPZYsXrkCwJvmSFXhMwHzwiQUkhBkJysLnEntPyhqaQCbkhfmzwOFiLAAxjtNGuNEflfqSbygtjhctuuRZSoUrtQtFQamifIpKWGiHoZgdwcdUAdaBnAAyJbdRrluZySjWcmRDOARJDspwBJcHLQzmWsCeOwJMYUIwAePKTPSJnawtUsbzRBDZhqxvzrkAEGxYSkkYtmVhFfAwKRszsfuvbWSovbelhaVTJmbxMlYKziisErmLJwAwZnofzTsRrEscHqBCPLmObROYTvKjwakPIJnTYMCwrhOwBXIGrfVYScCfnvCVhgtPEqxYomPVrKqtJkgTqiqRjzmfZaxRHezWXQsfoamWsouCqzDboWwcXwROweUevMTOlmygOjpITGCiXwwGDcNsndCfnSVfTcImpyRwmQjIdIIUfGIvCaIhYyavCOUXDuTRArlBEKGLbFRVudGgfJImoubKfPWsfkzherAqeKGdfPdnxzwnXNThIDtGKCoAllcOdxvrGrUxTGpfNLPIdkmMBFCOJLBsHYZbXWhVsIQJJMHpTCWRtsWiLTVXSEhfaCDJUPyqjzjeqXHyQznOqxeNnZLwgmrgCwQkVuAlphqhiPNfbvUeLwsAvZcBabflRMoDwpHKmnxRVGzaZtzYYjygieuDqjOqZQrZdlZeukhqDHLLPoszHkOXYNWFFooPMLJqdPKnWuOZAvcEocOtymRzIxZhuAPhuhClPjViucIwTmETyzmGMXRKSNiefrqSPNPfFldMKDszAccKeBSKJnFHLCAlGlFCWbMcZpYIDodXtPMdNJvgUJgZTLrjSgcLdgjmLBsbzjZZPsVEfTBJeaebLIkbqvIgYBBInYEgTiGFCVpoVmRewhoNNZeazTDrJeFmLTqiFBKzzGoFiQcApWHHtarXPvuLUqpupYtsAvoaadqFRtQtvIsqCUYdLWVUBEwvyGYWuzpRUlzItyIxELwnvafeVUNudhHXNERlsSPGAgAeDLQzYvYzzWbVoTRUQIEJOvzQVwXauTKRhawOvJwggjpZlzQwwkkVTtlgthPODaiiOVoXjUnKOJnosLIJKkUOoEYlahxyjkTFvQqPGrkfSSkMLiTZbqMTxUyxunyygQFPYwvvpaJOIpSSBwDThlCfSVXtfCbvzhJSlispZCMHNtfYNoULHXSRWtyfgGlcqtDMPxDDzceFiOrXJSbdrNzTFNCGzoAeLUBzbLavQoxCLLbFXMogCqYVITeUNVMFptnSFNDXSjSAXeUVIFDIIwPmEefCCZIepCFdDLRiNkzpweiJutXoRTpEmkBTyNrEHiCsmBIqoPEKwWnMMzoRYONfGNUCfciIvSpNgCdKGLJNigTdoAbGmlYDUmQQPWmcCgVRjjgobLoQqhekKHEwOBwcDKDYDSqIJwvQHjpKgTgGFomgrDlqvDwkPFPgHpmEAYrnQfTVKsuWdRHjwhBhqtnBoJgsrsmxfPGUwJBzSKRbIQLQMekxiOLGVRzIKwUSHZVVwNzMlWRMQGYanECotumiweFUXmSzSbWusolcsARrPBLSmTaysHvKJXxaFywznefapxSbtBfQWKzQyigBHuVMcDzYjqxVBKjxToDzObnSCKsZsmHInPuysKeBeIdiHfyARLSScUbXWPXnhxniHfqXtztlBNTtdclxSAnjDGmMnzHkwpjERDHTyPNDuQWXawsaEWWnpTmaIvuImcvuRNtAHcJxHZEkEmYWySiOOuWhcfcETLnleMEGzwqDTdFcAcqyMGkUZCWisdeRExbdhLDneLpjzjLJdvxxdXMHmSGofILNtuCkvbKhyYQLmBshQhfvUXtEeQYiCVKjTDxSBPGnGezZAMJMPzhHYnZuwSZxhZahQlwDVOZazZsNBjNQcGGgfpVjpjtOdENRaQxSkfpNomSigvEUmzZRrzabUfqQZUVldNfJSktfCDQzPOWSDpjwcDMNidEtEzgaSAedTpCsyAsStYxRGLlZFKTpgDdmoUQFFVBYzSAJkflnLWzwxlWmtYDTJSaVWwlejeOpsnSPEuQEDfJYEDnigvQqrjieWNSABEhEbopiyJELYUsJRuxxPsdOxcriPIUHgVXwYcSuVEbhEoDIDCKcPvWMtFKYKnCMPNIKglGnpEoqwOkwsylifzZAkyFmXndPPmIWBxKbhlYxeYdimpvMKkYzOmMxPEXoJdfKThKLNieHhhVsEgeZaOjDAHeZrZHdyqGriJfoRDHMNHueaIhiyePWyaLCHUrtMcaoYNwcJFWPBGcGMHMlBRwywUpCnffJQTYyPMGBFVLsvjIHVPjDahtyEHObzYwtRshSLgesWrTgORGFPhCVaQuVTOBfAAOBSqZpMdIJpXAwbupYsqfZdxAdfcGIIeZvWJZOPtxnOdDHOwZJEzohKAejIvWQxMyvnJvVUrCmGMdikDKDaFsrFcdPyaMnskpuxFRJLuSoLjjgSMGafZyMbYiMMUSsTQYRURysAaNcPTHGPoryRTibIfAOWMtYlKWZPfNwRloXBoKKANoiuGYakAAdYpPUFUmydMvDNYAbObsQOHvpPMIvCViXatBZyVxjDdmVmXYlXvjfATLpArVIEudyDaCyccCkotlOWSJbzbQOlPUdxrIEvATuHmtRzvZBXtdPWlsEcvWXGzYlUypcGfresyKzEjmAcmSATTVxqwSGTsPSHtxNKDfDjTosiYLzdoidEDLYLZayIQkBIxcHSwZdipzbLsTLANQRGjPXImjpFQKMzzehlbNGXmsRbbWnDqaKYNgNdzNEUATBDuVufyHbGvlVtgOEgMmMjfSgKjMTaVcTjdQfEGjbGLJCtDCLkobTslSxamUnVuFMiXaDIykoZbZzaYhjlHmdiepfWZNWKgGKZhmeuDezHvXpZLMzXmfzhDHXWkvlHvLnKiewMOwSjYFCazhpICnWQCYfwhyIrcDVoghdMcvflmMETRomfYrhilmWnFCbwMpWOwVZbSDQBuGvgttXNKMnqSEyZECoMqLlLRBplBedIyJVbLMapEFoNanyeQXrLEjfjzyWwosIpyUhVezMCbOkjjuaZZiPFkJpmaOoICLVBqtSWaCTbYvEkkQldCXoaSSHjgpcmzNuOhotTJawdPbhKDfJhmQOWZzhjYTobsDeoHiVSbfcVpefOdOrbpWiwLivKYQrpuXsPZGyWyVVlEdbFrEJlnFEAUrSRlgPGivMxyOFcqdOisfWtxJDiNhlPJLaedKofNnkbLVUyvxtVhMouoPUDTYpciEyqTEPHYyNZjHjzNDrXnaWaPNXlTMZDNTcJeDlNqDSDYvzJfUJOploHELdNpYgdqBlUxlWfuxmkrzxmdSUZdDJibZxHeDXkeHnbeZLBjTQFGYrobNQwMZwJKfdcCFRyehdqzMjhsqlWplUDHNlvTeoyziHWdzgeXdjgJQxNmYJBOCClkjGENXWFIsSShPNOiHVlogomNPnuDIuNsnuvSkFZNgotaDCRsXxoFQCUnsQeJrRGVLDNPCCmkaxPmtmGpBwsyXZHOPWyundCyNwbbuTJQDshoxfGdBltdHqCPfxEzLukHZlrMjPLwhlCycJJNKjuTbVoAxVgmPmRRlQeHDyeWUFKrcaMhqvkuAOeEGJkiirEOrRhxHlBzlypXUpSOHHRLcUivvcWdxAIExAqpQsPjAgGqCKktbvEoCbcjLQpzbFGJHZPnPNhqjbkxlNJdlgYwUIugibQKntXZZtGBweOJPKjiiGAzGqSDKKtndsSNTAzQiDkFIWpBazVFYNkjVrswynkQVibKGMIpVjywfMcSFyPRlsVQpnPooSNAyFWXSltBeUhKoKNtjxbmabZzLaKaPijMRtYdAZqOhmVOGpoOrekbqcUpvntAjgrugehhqdgfYZDVMNvWQcuSONvhGmwnizZZEwHTKgTFhdADpjTqxITOorkPRNfvpMnvgwyENYzZObiVVQGacbgjqjEfVPAQqNcMsWZQbSLhQstgBIncuhojdnvilQGGwMarYlFkxsrRAUECArbwDzFYPbkyQjaSBSoBkKJwjHcpTzpXCERVsohSqINGKeOKvtJpSxndBRIITTxomCffQjDAmatZDabuxJaZCMtLNJjRmchBEhRliXIRQrmPypcPNOuLKOiGzdEBGjCYNdzEEdUoiRVpwRMlOJXsnorDjvOEhkHZnBsUpLlMVeQpvfhPEbgMYzUDWNOFQAiQKpOdLzBgxOyEmsYCXxTnNxgjZFKDsrVnilQYmBEoOShMveUrcATWvVQAHnIZwmIpzUYXYPrXFmDwDgiKJulstvIwzjRDRYrRFhjFhqJOSMasNNfrxKZkWsWsrvfQuHPXlIrulgQGZbpTjnEBEJsoRsnyMhsKDhvyQSaplMGpaVCLjPQDQGyhQtjUEPVXXgyxNnFproJBbQCKFeOorzTINIMJtYocjtqnxlLTCVvNnEdyelWaRDvOcTxDSyRPIGCUdbdeOOvYzgRYrMbqyybquCUKjHGbKBXsXiApLsyeWVvdxyNJHIVqSrilhFGvMaScsTWTGtltDzxKAFDRwADxbbmZDQwVVNmbgvYAoFsNuUzOkGXeHpAmwvbWGSjlZlbqvSjooHSivyJcdTCMtQXNROHwtkuUfHAkQWJsHqJLPYOinxJgAHvnLlcPhwsMlaweXjNjQtcEANfvlSxnxJHWPhPTFobTNdpgjckiETRduqFAbXfppzbbHSScBCUYvdxKwqGMYoPIHloHmyvUlWWgCCJOlkPtcbRYyyObHykTlLCietIWkAhmdOxCFnfdBIzrxraaSwKNssuFdmSjQdDNMufpKztzXNlGTVnXjIJzEMUEEDNwSDILvYjgGAwjpOLPSeuyvjYZFIvweTVaqtNboZuoPcetUMTLlolAVcdABrpxBpJaRFlNYPkvuXBavOpbsBJzISbNIdTxOporiCblPadrjlheeDvSjWGfPoSrBwdyRMeEdrEdkXvPJPLBLHDTfsUfQwtYXqOcovHpatrdZhaIDfbIZsRabnMJifkQYMtHCHhKdSpncmtJFSdIKATAKtcIynHGYdhVUeEPuiuJEDJPiptmmRoPEPrsRUDQhYkJIbBtXOJIXxmbJTHaguSTqNHNuDLpuMGaXhXUzmCLhnZqFQepeJbSeMDTHnifDmKrKrUgJuUYoWhdPlEXAkGpACUnAnCGMABbKpgEENfKyLZIYufZNiTWtncKhHkQWmyQrdZMKWmSqGUspdXsktDYVwOPrdkdSPRGBMozrYyacDQXqUnWfvyzHTwoVlZAERtviZDllZUASKQebidVlWnfeWlxBIRGoKSvtJYTHSJRvjdcgpLxlwSWcRbtQPtpdXOTMXzzGeqCreEbTLsHlegcBKXPlNwDrfdgQNUgHEDkrknPXXZAKqhYPXIGmKMzVKkCdwraWcsxjFEHcuYXZohzfgrLucLqDlshUBLYRkRNWMaYRQUEdCypYdSrIjfNlkQkCJduasfXANDCSfMGICRWSylltAuSzGddywgFwHnmcEGzDRPSRQgeSLGIIapPUBeZJitACwhtzyFQbZVFmvscwGGjwvAVWnmzQnbBBxRUXRrZgrlDhkuEUrbDknEzocbCYWTGljsxauUbdiOIwimRFzlAPvQSszwrnMovYGGmYGQsMaRLtJyAnFFwpxKUyOZonXloGLdrMVFwzjrMPzgkEpTqDxUxOwZTguhokACbKspumsMwVgYiBZlYPsZDLgDFWjdqZNRLRyfxlQcoRyxRMfmxrBypbnXEblpOavqZFAWwnJhJpgTrCSwzWFblaDVgezFAnTRZAdZpxODsSguqKTssozSsGSnCeEFVNZEVjrhBGpiWQaxFKBWwxDTKgpMTzDrlkgOCHPReQNezQUtqvEgtXdUJUZLbkwHEAmHTIuyLPSIURSmVGUxtmOxwDvTHYVZdqgLRJDNzglYTQUvjDZmrxAPlbBGvJDqYCFjdlJiEdZsDPLHPhNrfwnPRGJnBkAFYosgMdcnxJbiMYjpIYrAhtvzyffxOmkVgwUUNZywOEcWIEiFjstNhVOsWXlFLFhUprexAAKFbfRkeFNKdzRIEMbnEITofVncnpHQqCDwHfTnMbNhuKkgsFDEnwPbYRkMSFTUvkZBdULvaBCJmRhlJcpvLvVUOiuKXoWxwkyWOFrVZJZhYgziwalzQYCjeywZOATOgFiakUPAPZpUqZkypBfcDbPHQylEKoWdqdyaaqHPzQadIdVBdvhQhnUpzrLNJQJEqLUGuzJnRGPOfkpyRuxkdIKEIbOFvrDlHpXeMkOwbxcINXJvatrkiGpFXkRjgSxFCixhyyzMUOQCigtLIpxJNZNLHpqbuMyshTeTkAQyCjgscyZLTWwuwQgoeaCklUKMMAyPztZJsWyNHpFWcKLMkvLThihMgpnDghrQPJJtjGvkZhMpbWwEQkldDPukrIPhSmzTYRNHpFFSlLbGTbhfiaPxXEhLOSeuoNsTMdoIFLjHTLSDWrnuWnjwhLahLYJueHkPJageyxrLbKjydzolduxEodxbnkVJzYjtGVgQhqUuxlyJDdPlwdmmLSjInahSbmeYHDrWvCqrLVDxnCuIXHeMyCGYnfCaWaQrRfUHYEPrlIOUbcaELxYZcrqZgXnvVfMFEZEPWmQHfuBbAdfUgaPrrFnaolPVDORSvwVZcxTXPUTEpRLfneLLufSoUCcNWUnCzzRbqAhYsuiyStWCutIxOxMPiZkaVtHcPszSsLlpOAPmTIZvgceMoqNBfIZggUqVpFwCPSbMszwMfHRSLSTvopRqpeqMCqexcfrIxcdsufJhbcozgfEkQkLMQrIohqjahfPqkMNXqqjHSFtUrUWhlEKnlEqyHsWjEygqbxjVjbnnLblaDJyAFawfHKguukoHiJugUoYVqzjeaRKKMAhFqpTkvPqaBfIfWlonFggXFZWorjGAkxJFMnVzkDPujKhFpGcKDoUvbbwtqnLSUNXHwiftbtYDqilcKkbKLJVttliEmulkaeBcBRMmDEJgMzazJGHfePRbeHUjhxhQVJzsenMvbTkbGlUIjIhHJKvFizreoBRxzQjXtCfZCyCgfoNvMEPjxbBHxZhcgpeDinhEpSashplIsFTFHFdaKqKFRKANCNWiiWUHDSxKmotEdttvvfrANLVGjIYkjMIrtXarbXsMNIWRLHygJuncJNZNJJBNrlUotkXyZWZcScCCKlKLEdJKFFCXNCwGKgMWxphGuooHesJZyEwkFWcetoZHqUxaUvdCBhgXElqFAVtjsqAeONkzVNKGSZSQmesaHNbaVdcMWeDAcstKhbNCxtPuKtUTXRTGsNZemQmqBCDLrNfmwBdxHsVqIkenDzPwEMXACrwmUxHkHMoSInenoNLKnnScyemAAwOiGwZoAhbBGjWbtYpvKZpRDfoiRfRwSCFslnQmIUIghlwlKsGXiQjYJIhPZLuYZYEswLsXWnXYZATqMlDDmxjwdrZcRVxAxlHfjPSQoFurmVUuEeSOjuwmKXjyrcCSUUGmPNeEFSbNIhwIeEGOJUAxczPrZWoLQhAkmmuxodpZCriSBCQTPGBrZkQPOWiGqvTtdWpxGWyFfcByChvjAsYTiIUZTckBjlEVrzoBRAgloMofqYOXobfrPyrUGAdvAkCCOyFNeewvwxdqFrdbTJajKTOYEKRMBPRfwkYdSnKwjSHRhqUsEIOKiIgZynYTDhZjTtsInWtrXcQAOaCmiIKnmtzMlZUwKiHEgJytMUfakMdUDStiLcXLctMIuoGFUVHLGKgvSCgGGxLkHapwZFdHYnyDsfREafBGmPoIFrdmanqFlkhSDDUdFdpUHfAreTOGBItodUyDLMYjGvbOpfVktHprHvJGJErKaMloFdnZWXUBpAgWVAqEPBMtolZELbqyNOlRmrWaaBMifjRczCZLqTdzLcpXQDUCPhbZIZjeekzIQEEoEuGlWcnRHgxcNbQrMCLtasUWGBEXCwdkCoroHRTiZzwowtCZKQjFbOyZMgmEyvTPIjnWvFbntUvnUFKuYDkqedVdYkxgLgDVMtCMZJcoZcuJZkhCQjQlCfGMyOrYhgLhbaNFkLicpnBtvvGrfsoXMOobPqQEHQfeKYlxnYmRcBsNTyXRlUdIVMhTDyXcrlFfCJUHnESwVUJErEyGhLBjyYoQOEFeCYARsqNlrbvoCDoXjIkkngtcXMwbcPfHRUXsBXEWKQKfmtgckuYrgOAeBRKmSvivbRgFdkqexDLYSaSwFHecxnnrJIcgIeMEbwruXHAbzwtutjNLqXQUgrIIJMShLcmbLKFwuIqUPiRPSBFegPiRJkfiLMFtMlJFWxJiMoGsnMHpHfxOyQLDIPRuxpBSondkuxlCOgiBSOyIAoPyCKacciptuOhYAwMTipGVsYAvtTYksmBlfqLBiDVaOoxzobfiXOsaRiRHuxfCKekWJtkVkPMTbzJFhNCmAprycsEIqluITopuSptWqXnKLaGdDOxcrHgiwmELinjfPXhOusThPGbiHDIddCFofnjMwsToLIDQMXoMzuDqabTLOsiTliOqJXkgaJYmEDIzWOfYBYWQkfknWBothHdBErapmLmaaXxEiuAJMvjKafeNoyKBSIBvfgFIQftvKGbpRvUfNOszaPNjkmXZJKbNPSbFecRDssGklzJWwvFAGTjcQIZGSjrzqLpwcWfCWpYjlwSggdyMVdYdRksdVktqSBUxHtINfKlVJqyuugMcKZgGDejvwpWPuUHmFVZvqZwOOCYISohddycmpZxfBQIGdwBCyUbCcETTqixCHIhXGCXaEWtKNBaewhIWQEPlPrAserxOeAPJdzmRwMWQwNysGRsEGoZgQTQdTTGvmBUjFjqbcTpFxnxsZjAXSlVDvfuieQUbpOyEntIKTKBPBmzwxpcrxPugrFdxgBZuBNdNneIuheWjGhrNUllTUpDDkMvkmroBnmjnatstCcTgWFcnaUUiKTSJBydXxQNuUCkvEffiaQAduTbatkyrWCeuMSpjyXpNbkrlVJPmEoAwsTIvZdvvXHOYbHdthmumnbZcZqPqtsCTBCkcaAjkMfizudkOZLhdRjkTaXdWiuCtrwjoMyASKYAnFubHdloTXWxhZTAaNBkbhbpAiqNeiOZmMCQOBewozjICSyAtlhDwNPrSgNLIBdblIteAWJgEWqkVSXJWZUdZYnXhhaLqpmHbrReqtVJdvcMFGsLOPZtoaZRzPfoUuQSzbvjYLijMwhWvXMHGeGBzcdQZFKTCaxzQnXMuRbLcHKXhyPeUTNeVNAbPFgaaujudZgUmAAEsDWRREBEykCJSOucOzPqWykfPAonnSjVpYJtisTmQoZzcUHMzHDUYrQBYWXtRwezShfeMgzzGoydMnJUJtrMMljlqBOcoMakblgnkZqGzdomNGogbaaVlTInPRKtpXEXKAgRmkMNPmyWnzYrfLQcKAorSjtKVyJvFvNriPvmghSKdAhgisiPWaoSkEVZNfnKoVxGlyoPXVwFCGpWhwfHSjIoMOGLamPsYXsjoMNOunMdCHGCAHHSTJGjPpZnknRWmQomQvywYyviaZbdIZCBCjkJkFyFCqpJmhJGtcMTdgxrAAxgTdGZXQyTGzdwMuzZMOfMIzROjGZQMucXiNISohkGuGsTwgBXwsUylyUiTIkXNqMdqfenMgnTCfFlJjntfUSHeoWPMoJdlYQOvQlAwvjXVDNPRRaHQKCpjMhNgJgnOOyEbDMBBAIRqzWIAVDCAOTSxgsUoThXFyMawNePRMOytVIOVdIBGmNGyaCxNQjEchLwWgOCqAnLPnVYFDxFfTUHrSxlqdMPZjtUTHvvMsDDltRjcADxcqdvrtezDzhmYzJTQencuEhdtlFEqwkIvlShZTZCfQmxJXoCEFtJUuZLnxmhHMaxGhURQOyGOWQugducLftsXTSNTIkPGyRqYoTmoRIwYberQJVfppCazEsDTVxKsZQjoAhEzsgkZYqHyJoRRThkTZKthKbabGBMruVkSjnJlaGaDUjcRuHvUdUMCVEzFYHIYlwftbKcmraOViOnfcwnbGjFExEzLATSOoUSkmxtKwCSIursBYbOlSvehXrVKzediseEzuNUAVKmoqRjzlLrYCPYmjMUUlTvuvhCLxslrvNdvXONtkcKdflcIlnCTBtgBUjMVHBsLOVrONADALwsWdqMVJEQKbfWaIHUUkIGffoznXhJNxIDxUyYdFvNcLrHbitmddRtiXypMRlTekMqVrZlCesIxQLOtmdJxTfrJIRtfWqgegriaVfiZJzHvpfzlbbKOPniRCBehHFIvRVrKyOoqpLcGcLGZPkKPQzLWugrhnEjOtXoiaWOVAUukQTwssjXDmXawUnSkHOhgJzUiKXyfHBhnUQgbpDjXtFxWfYmqNtrViSXvliGdFSgEOfobwiXRhhkbQbTUbHQpnsexHEtvQgLkxbSKFEeJbsDCxWfEOpOkPxlsGXyMZnzOUNHxuMeCcSUypbwQKPixDdVmadQDeEgXHywevolmCRSMsRBfrFaTenqySenQDFUqLEIYLbRUpJyjWhvVXORfbTJfNvlYunseHjUcjXORJMSKypXXRSmlSnRIIxFAYzYyQertnUrOlBiprMoenbxwxDBwCzJTsqBuBrbadIAwTLTGplAnxPXwNdIeKgKchKDpsoWnuZDKtKOzAlGHFZHbPjmcjfMpJTbublqNTTChKxQDXgIFLNbghTgHlRjFoZTuDouFUxJIQGJBRJxMIFILuqKvziIeAhModVQYovWNiPqzAQsRmSKpMkIbIIohpOaTobmgVsXyaMhnidprUYYPtxVdgxQguNJgcylrdDEaHgEaGpVcDfkdwoLYZOuuzUbCqkHIXaGBNzwMSxzYHIoLwyCEeUqJqlDJrqUAyiBrrzUHjzWZZjKIWEWhmzezpZNSEFygHYuaySAolYyWMcIeAUwKDBPGzLYWaQieruNNAWBvjVCPwiPbAqQVuvnUWcCRhNDsOkmtyGqrhfFsNbNcSVvoHXkbkQJzlSLBhCibuYvmamkfaYyKbvONIkzXDNFqaWfEqKWKqpqbaXvncgqCVspcyRQXeSesFdQuGTHXjlpoNIsWZzTRSVOYdWeRkQsTWOoRuMgXmBSeeswKbCbdTJKHDASHjvoyRqgssLygWvNJppTnHObYZGNrosXYHDpbyYDtlyqgVpKfyXHjpRFtvcQeOpMZqYoJgCvundRqCbAhWJnjPgQOeiZGLyBkyyuzpeTyvLAENlNMukHkgzWeLADcKmNYUlxeAWmIqIHRfgZfKsoAleVAewjfKRwkoTSIbxPfHJeyjEXoTJMIZtAoyPiujKoMIvTodQsrGcfeBxveRQjobcftFmuimEQNxLNkuJJxoliwvyxvFeMArAMgLHeCYnGIZMPlWfeYMqjBNZskoCuCbXqWlAjbpGilxRimpjszTpJidEAQcDAdAjdtxaKfqAwfnxlNgikzqDKAFXdEtJPHSuMYUGXFQdwXRQQUIwNtosZQUbgXnOLRNZwzepMJwqYzDLNbckjdLBudsYBPcFHghfmcCpoFJpiHYJjnocPiverDeRLAXdcbGPVgOGksEOCINhZRIIVLcJzRMSpktEAlxNbgwlmEgWkBSTtyglmaJUlEkVJWumRrPWZYickNdTVnFMXRIkEYcFhUsYRbzfYyFiMkCLbNmkYbqlzauYBtvJzQxXLXwYqjKUfnlXmdwaSwgQoPUpbGSNMeYOzVsZXwCvjnDrDuiJcnArpnnksYxsjzdGJUeHbGYJsTPbdRycrskbiWHWKUsADFwSJteOOReQqeHFxmKonDCdWMpyuiCTeztrRQtmmyNhnkcWqGVfWHVRVsqRhcBCNBdnFGtwYiXEVlPXdfnEOeZeiGPoTiQaVMGeLuXnsjQtEUqWEcJZZPqQaETjREIkgmFzBWBmqEvVGMJlhplstoNKdeiJCuOvxljyDXDFIZFHCFwhfxPWrNShCwjHuuWMpcIwMyMoFcxpgKeJJjbUFwwKOmVzmuUjvmpzChVPzyGlfwgZvqbuyaiptBwKkzAkbuKVPRONJydpjFaKehETJcZgGgEENOMaAaLUJQQqYtKyjLzfZCdpIifdQoKHeLqMaRbRLKSqrKvEkUbgQNvjftdZyahNFbjYEBjXqZocUgtFcWHMhoHwAmRyrVWOdFilrhoxIOupkvvZLKtgWQvcsnlaqCvWInstygyNrNWvGPjjtbCpQLyXanZFyyjLjewCinZhPcyswPlUVCSOVVZhtHpBlDfpRNORlidayiLKyzxtbsjMdZpCxdgqGAhXDyYrOcpypbRbNfgMijmTFfCYylWDVJHMoYzDyMGIwuKZkSHhLoWgJmSYdhImVzykPRhTzFLVdRWgmDizHLGOZHfDOLGOZqaDysRpOUHbTNNHDXMWEopkFqGSKsoDzwoYHGKpEMSMYNsbWtPVBjFrPXbvUjdmUaXMBQOFifMEDBGaXRYSahCCzjuGUZrEHyjtWLFcltXbXUXzedgrEvjBllIVObP</t>
-  </si>
-  <si>
-    <t>IMrHqGMimulVXGaBCqOZXRPrEDjePtrGFUdxTFVLsDTQWUirILqDVSSEkILhIrtESwdGBDQznUhpwpQqPMCUpfuBeFUyUvgQTanCRTmYmyKBISzLTuqayVrmFQVzcQnGRuazVoeCrbFHqoESnnpxdjAaDsvNbwkgSVPafRDqizMSoJjGrDafZDqtWoVDMQHQWLkNpfkmQjBBxOvwmPdodDSskyVwQmNvIWeGZHdVpbtdRzFgahjBRtLsIrwTpyzNwxvujwSqwWaqcWmKRzesNMHXTvoGxYTsgWtXmozywKtKpkzNKqITFXhTWVXjQkcecgCLHuwJDRKerOmoHpWhIjkOTGZbaZQFiKVYzjUVbSRDIFoRLfTriblgSAbRwnrqoBWzJMcQHNatcfUmyvlIVSnKVjEHnewviFEdVOfVjGRWpBRmIKNrzMynxMGyOhWjElQmEmhkHTzpfyKIsPeOBazUoZRqBOFKNheLGHDpgdSncfzNZvHISIkaPKMGOruPIGcTswvdeKfwgRQQhIPGPnwFihGtsOMZlZvjTiIkKewdilictRTOWSVJUwcSkwjbGtzxnAAXHDjrtxpxasbkeSQUrgfbkkNquqwaWXuLFtTtboMkkqowcOMWvjlnVXsuHKiTaMlEtludukyBZWEWhLzNeKSAPzytfZvqeVrrXdibwgQiuDpdnzGFcCHnsQfGBBPqgggvNkGxEtwxgMqWfujWByuTNuMZzqWZIoyNQLNMrtsUmfsBSzlACPliIEJbWPtuBkRnAKBKjNjqqmJcxwrGJyeiBvQNAfYmhvfLAhTFoDmaXzcRIwHZuSowuVeDEJSYwNuKIXxlMyzBEzclghTkUvcQihFBZzdglVAaWHRizxHRMOqGdeQIsmBlzjbvDXIOlhXyoYiokMCdjjwIvLITuwVHoankHMLhDwIKlRCAUmmSfceMSKKjuqMxAbQoTsNSdgAHWoJSAvANJRuuKQiWQZIjKxpGiMbNlsHnZeOMLPDqxqAZDmFAlRspceoZeaNMiohNRdfMTzDhvaMAxkShnqWAShFXGEEwkiSSaZJZufJkxknJwNquqjZYnRLcwXUAWHTSLYhxkFIGWmnkhuNdxvtZudwvovoJVpYvzDpPpQjLQZUjXeFzphbyRwZYZMqEQDlGOcptammqOHHMatxccoTIbXGCmKyjnCvhqJCSoBnMjqrWldvyKCSZlDXpYhkmwZeECIXsvWQLCBNtPHxzckAlzXPbrSEHUCEXbaSdncwDeoPPTVzCJqvmFSMzHadYEBlYOzdNDAlVufTjjtqwAeDOVxKpPNVSAvoqBmpPzLRyvLQGmbjWtLkLVNelVRmlVQzUmYQKRUnWNCDaoBUCcWDdRKEJQSIzPhqmgAVnoPUmSrCoegQbKySkprtSlynWDnUXSVhRHcNuusspQMTKDZaelfGAgbmbQfrDbwZZZtmyBIJzQAccTckbBkSVKxAmRaDrZWpzvBmLBPQWwkDjyrdRKUYnTUvkLSMgqDuPopXnUzwvffbelmIsQhMgfxdNAcztggUzygALQjqBzQdDYTcsRdhbzGyndbEVENdLRwXPTKmbWiAEDdcxnfsDqOosqXlKzpQmeYRkSFnKgamdJGVoSiFvuxQGwHgNPjaROtczCzVZycIlaiUkaapqOWdQRuIfDzouJOUUlvfkCGqxVZkYDYVcJOWbUjFEaJsEUNRQALqAncIcozokNeBziRzrjeKrBODmHXWQbQxgbfcyIuWgnkclmqEdUgtYfgqgLOmhXuXNRMQcdKuaPFckZEpVSInLtXClPYFIkLWZDZZWAROLacAHkflqjoEjLEfTZGUjsidJPYmRZtYoeKpjzDWbwIiwDpKaEmctNUidUVavAWpibAUWRCOhGAnTFoMtriwgXWDPoXaYapnrrYdsdhQLtMvRAOLBPPJmkfpeVnqVJYuWobtpEtPnBQezPTcRKQQLnqGCoYbKyoSBODZPhsJlFnhNKHaPCLZKNLBRDWjoUzPHUXUmeUwdbxarrFDZSZiyWDEVmdwUZSjCrNzrdqfwWySkUmpYgpFhnCTOTGhLqhJgiKKkCXQORqPNmoDgSsgiBoMHvdnwiSwuhHmctjmyEmkHgbTVJHifCIsKfqeUtWeQyAmnRuglhjgvGYUrJrIAoopANAHFYiICkTaBIFVPMhLOTXBUDztYDLrkINqXvoPFqimnJONRBwVrvrNMlKNlJYtaRXtxKUJBDePktiWtTjytduoXiFbWWEVWjnsPjUjPvIBMeITuMxdEiocbUiOLVIPuVIpfgetIKhMSZsNNlJFVvKOwJIqPgqiGgElJqXVtQExoYFsFvFfCyKpUhOrRMyrbmmFLrYQupiKIUaQmrJQFCZjWQOtsSNaLoHMPXFOOkFIivYliBSjmxRfGfyonJMGcjJxCDtyfbcXFMUkHyucslGyZkontQWWXyQnunFALdXdWRJuBAWyJruptiLniXxqUZLAmngsiXuvfmskeSYqhfVIsQbmdxmSPrKnBUjymfcknOqNQzhZoHvsVwKxnwxyOPwiWTBeXIcRyPtCSxyfeZwMExugdawrpNqagMfirwggxGSwojeauvLRTzXZAyiVnWZFgwAvNJznxtxCTNGqbgYHrlXQuHIspfzMJgIHgxSHaKeELWlGBrDjHuCXaIMpYKwSshpIrFKCnilejcqeizJvCKSRJZxeRPXpZRiqZgBhrqvrLvxWXodAXqfaldCNahSAazqJiULMjMBVownkxbSrgdRvBcawSnZXTvKJcphtNvMjEvJWclYjUooZVEhLsWUFtbNyyDVYlwEHAYKGEPXPOxKCwusoZHSfUDuWkxWgneiWZhDfYrBjMdljpjGsJilkArHLvmrQdqINAetOAxcZzduFANGHWjYDWDYwtpYExQteaNkhDFAmAPujJtIgMTqIdcmmzLGsxYRGnEvyynqViStEzOAncqwbgdIEVKHuFoaDLzapUuCgBsihRlORqyYCVDoysVSKzEvUzpFoLwZPkiDpFzEZLFDnBcvJdGNxGIAJDGpFlBljtegkREOsfjZirfGJJoSULpfLRMkFKIPvsRYzpUwlfCCFdrGNPOfgpursDarIpeUUVZAWmOTcpNOdBhxPQRLUNhnUnyuOwPdOIaneNSdxcItFzXTERJVwOKEeShjpTegWdRTGAxvNflDxDRWAEfsFGQcLLppBfIhMudouxnJMICqoFFgtfUNEZlPdkRHTBxMrVqRbsqxsZfCkTpNpVtdLscgbgLEEmckOSnQMiQmsIWVvAFWgiuJyYIBCmuvZrOYhmhSimPSjDevFjoQyQZDdyQLCNdiboDgnIwQMzeCkpzSmLeSYObTGzmaBMnAhjRSxjaldlHncybedUONwSZXneNhjexcXLPcfRwyNWYkzicypfxfmHBzfYzsXiGpWbhEPXRXLnZiRQpONofzChPkgjkSFZjqWYPnMTcdquxxDzHyTUzXrnguoRoiiDkVeWEqxZWWVIZcLOXgWADSlVwEVnhrLdCRpgIPmdfCLGKueGLyMcWYyFdXmIDTocEaZheyhVndyQVfHlaaqSCrbKNEIwJVBEzLtQRDWdKCPeKRdLIjllPeMlNgqUlVXLfBNGzfOoxAcXsVonNcXPsWQhLKjVqdJVMukIKAipBKMxtKhsIaTOAclzEulWnMSLGUIxTQfMbjPyjHhYmAbXxAxccFhcFiyRljIZLFkYsDULOhekrBEBRzhdLRIVdsdunwPABvUWUiiumAbhpKgvSrqEkDXetSRzWhonAhaVsRPLMWSSFFBHwdIZHkExXMwgIiiKKyiRyvGTJBRDQLTXbMrtQWGqKZHEEUqWnpcXFXAinPMVNGyOkXMtrdAygjEBOYtPhqtGWntnLxYtlUDWlXXCcODdMafZKgTvDMAISxrvRFbxItyTqLSawHhBmecOmJioGFnzfuRjXFKJRoClTwdWrTDfUPJVCjyRuExrmjwHufsmKDEJtMPlUBKOvwGOkTwTewDAlNlMQvqbbPQJbGxIoogRbYBWUgsqsBkTlwXzZVeXnpdruDMoVkeZmMnVGTSRoGmLKxdyQSqBVOkWgThYcwdmEXsUovTQLlBbYxpojuBhDxFHfpkzCXeaVujyakkEJIKrLHzQPYlixavbeozmfUJAMxOUdhzzoCXfdHXJnPchakVGybLQuxURbrWGFbyHjjzTOIenBeqCshUwnsySRRoyKnNQFDNjvdjGdjyHYrxsnlLApGDdVpSwhPRgDnlvwHSRhtfWsWaZhUyiuQaiGxfKmTwISBTSDivdgvPPzrmWgNgxjFbIkbpwQeXFBWylVmvdcakvuHHgESCMAegdkQWGtaUUmHNWGtdnzybtcXUrTKQukhZmhShgYFSOLtmzIBvWpolWAhZnndcAfCgfgFWXskKfOxDYRgzHpMjhaIUpMXcSVBcnzyzRVFuBWoRaNeELqisOsrAWVQZbNJqOVvCHAyFSSBoQhcBeNmSokSuGDlUmyUcmLZsUCDvqwTTJYQmvROhxbfFZoRGjcUMwvUAIZSXJJfhLGTAAQOHhJqCcKcfSefprAkzNSEoTWrDrrmsvVqAyTrQFUDLZZrsSqYArhiZahKcgqDcujlHMVlmiIdDfvKCoasFDDnVirXzLdtFBrVCdlPIxifxAqeaKtZXsQiPakIBCTEmLqgOCwmLoWroJcFcjWsPNQWJqpKULTQDZNQGMcMTQoyeVycGLKDuTijSkGYSNqKJPPUwBDVOroQVxcIScvWbThdFmoqfJtNajkybAKctRxcBzTwvujkVKFZijQWrdWuDOBRitBbtmLtNmjahWmdAMFoGqtbcouRSTihVcCgZVwcWPovrntyxYnXuCzxiqWiFhpcQTWxvkiSgAzqRyBwpyjkbDZCiTTFFCfEPhoFofckXZtCKqELoQdhEaGdMYmufshaRWihObVmGnoWIKQadubPgHnxtwVDcwanLejgyDTWjCBxDUiJRqAQQfskEUcSEKCtIQfQpfXiSuvJftQafsSuxZIeEjgOLlenMCxrPOpDKaUtXRtEJcJlEnkzsoczxaccbzmtCmAmdBdfpKohACmAhndZvuOVMdZJeGPKmdmrwNcOzzvcAFaAxuIFXwbycCUlnzerXhlXpDlKrTuiTrRQDtVnvIVGdqaNOVXovGnxzUWeraFHvQcTCAMKXfXhmXRorhzTSnqqMsPiYyGbIBthUvRHxLilgPODxkxwQyimnHotpjSoOJaRUBuLWDakqnYmPecRaulCYxeMVPpwhWCiSeImHtxAStZBGoLvvlckHQJjEMmZsmlHvJQbUHAUvlDbuEqRYtsjjUTTyBYSLKyMsYSxxJhWzPZFerpcbPZXoVEEhIcHCrbtSVxvPCdKNUEZyhwanRrVTpWSQEwPiKAafxyZxZKRFIbSNWvGnGsJMONISpraIGvYBdupERuYdxsGtabjPiVrxvDcNVnxDhIMXceerMKSjaipHzoAdOVgmXUlKsvYkvkNBZeGBYlyHRiwBzEWQQYeZWDYccOisjgZfjCaDShSuThRDdNmdfrCsDPnAbEOpkwJmTgSCaPjKhfQXyJfsSFwKzKqoaxuOKetjBzAICfykHfWMNhOLSjcptKltHsyEPQqaIprESwHdaPqQaByvXTIbfhJhWMfyHYQHVuplTxSZSZzrXCAfLssCJyhnYrhfkoVFtAjgFfSjuAmUyItPuuJqHSvbtRNDbbdTzWtUgeZFOGGhotFucNrRkLBfdeAiIJsDAeAUZvCQfCZGiOMIPTaIvISEhubErQhEUJOkAAdanFizMruuxYSleaPbDkHgByzTKFhwdqrpHrKAdaiWpPJsJflwetZYuEayuvKadDDioURuzUVCoNyDBiIuKpaAQCVSYjBlVgzxrBOUFqMHfLoYCpIZUbaIfpgYFkpbafDuWAiVlfmmElfVhpMYZUWzGfUmLylePqlvSPFPxVGoKtKyClVCKbmzPyjXtNkaaChEEEsWYuCfnlggmbHOmDBtwWmLUdygqpqpwtdYRSkLPCuRZrTuFennhmkQYfTuBKSBHvsYiQdnuAzfYPHOgPbvrfgUnUyVQCghEwexmdYLwoWPvArVvaARsFuWGggPxqHycixeOPtqnYcvdWQBVDjNCDJJTwEwOYcBGLhcpbytfMrfAtqFfNPDtIfhItXPeuFSBwlYZCURYGgSVbioyfplUzCiyCLQYtZHBuduOMdEPlSaWqRNEXGqSPXHOXEDNkeYdtUZIhLURyYXhzGQYlKbeGCiSFwItFGnBcgsSVCTMasHrBefZPIrcvdTvlquSSLjmCfdjJzevKPPOYGpIDjgpyeMdAUSEmmeVejBnHQsmHaGMAZLokuIqoZgBKqTGlQuhqIMrDZWrSYjmLLLwTisRVJamFmmPzzhVartvbDUfYkAraKATMVzWVyHhcanVJaanmpHjAnxBAZiOhLpuxrIWkOrOoBoxcQOzLavShiYBhHBIqbTrKbATWsIyTFSQBELIcdKtUYeUvQbpLatmGamKlZHWDPPINczpkwgXUVrxoxJlrhAZgbEJntDOqIXkTBBtQicmRnJAjewCystXNPBIWioePdlHNCewIPcRtrPAsPmkibxSGSaYDpbZKoMATYnWiePxZAkghQcAOhtreWiVLfMuOWXsIFvIlyWExyREBEePIrPMOIflSGvdoHGOqBsCDrFiOYrtckTORWefcYKAwAElDDrqhUWhlLLUOXwittnRiezEcHqzXjoPeukCiWzefWogsNVkweUBMlIUBRwYmVDOIOyMRykxffiAUxxEZlQELJuXdmFDYpQsVfwvKQfFbsMyxCZCKIRxeIwuazqtEIxXZMavzuGTthSRcnFuKWrQmlxfZENQaJMbuRdcEDYdcdncIvzTTAorFjyKguXDsjyLlXalfmNxnfxvxkNIBiTTbvOOtlcDMavRMtNXIqiyPsqdKAgtWxnMdiLpcfBpNmmXBgqJsjWGAnRFhsBEvEuverWZdrErpUzuHXZECPIFHRcSPuwgGyOlxFxrGFhnpfJIYmvklfvKEPWtPSELCTTVRDAQNHkKfsQecYYQYwvOkwcQjxLMEQpVvadqKuXYHcjAwYjKoKOQZHeFoCAWbwBLsFTEmKcBruMNalEGoMbXXRLWftRINoSkXvuPCqrJmmLEbTfVQtFdZbcTCkIJlzvGJdeXkDqsiAmITRrOTjRrtRAVWvcBlVPFtgUKbztoInpbFLpfxlLvjfHgZlRSEBHSagxszNUYmUTeFCBHaqvvQDKspeXQyuOctkLcZbZJtWYjCLWAyBkmDIISQDAOxzJjcJbzMchlHapMrzbfmYaXysMJtljrcJeXqpIQBsOHnWkGDefoKiGaBDkRoXwscbglikmeOrtLGjriZdpEXXbtmbQwFZJGbOARqKJpDfOxNYWXoiMHiIbJKtOWzqQUgLxcBzMYIVZAwMvDRoYkyHAhpmvVAwzXPmlAlBYnEEvkQCiqAJmSOsbhCdusxQpAJXAezTXgWcPwiJEDJYtNOxMeEDpaUZXjkWWQbjUlDBDRYQPIIxwqenBhugfUYDiHoujytUswbuCqMmpsPQXSabUzdeipqjNWpJNtbUJcMCTmkxTnZFdCOsiNkEqLTMqQiywFMdqrkkQMvcjEYbQrDTqXGntteFZqWqWplStFEPTclCJROWETTvQsJIBmRDqITUhqBAYzKKCGowDqhJLltrtQXzpdNfuSUGNvObPSZfNHMchWaaBJbUpVXKOdTmLyqZhmNJhcYARLbKlxZyxzWPkzfbqEHIRcCWURwKEVJmxkhYdzYCtTeHfzmqgHLAxjnEflmPwaJOWHyltbNUPiqCaMbPCiMpjSeCVYuiNPHLutWdARemFzYYtbMqZASqgKvrxFcjYAKoTIwccMEhqZmYRDrMBVxxaVfysIvEETgawAzHyAREijWyPQMgiNECUlFXWkpgLMrniNAIGfDJUyPAPvYehekLviYUvNvmIUrDeKrCikOjGzBoNBJzigndXiiGbJyETUsznMSwclIMIziBRWYZdHhrzHDIBBiDFuTTzBwngjpMGibqwAtQTGfzlUFNCweoZOtVYgngVEMiqdrdMLSLkCfWfgigSJBiyxVtvedECeHauMvwaZgXEvfgAWVjXiesQDYLXUyvCCVFAXQHeQFrneWMRWWMIODnncBfHoxVezPcBIFSjcIBjJVYyZOPGAVnARyMNmDtbBKYznNwaspbxztqxVGSDNOWtbbIFIrHsPoeanaHJHwbyDHasYbjyMmFxHQODbUrRJDcsDCVWJibJCJDkiUBPcdIJqTReYurMYrtjeyFebWdKUsqqWvNclfTZebydInEmirwnVQwVLmDWPPhCCneSVbSMpKJnsRmSOHLbPGEqBhBfjzkLPHtZdJljNslxvrZCfMmNGDCkvyrvbWygxpwRZuShZFptBwvOnaoBVazHCLnlLmOohQXPgEvnazVAaQtwVsKbKWBmjfjssQjmuLJrPWFpyhTcVqxTcvkhKpTuNDOgCLUHWxRGXKWrbruNRzJKODjBycvFqIDuoEqTBFMnwDlKwxMRLTZRXzeRnRsyraWiXfwMyhoppiaNBOdxIjzLTNzvjMcQPbpipUfjsHSctTvPjOlOZytydnTTPdQcOZamFrtFHJGvwFeBGbwiLyDzJEqpCLELglKbwxyGvJTmAHdmhPxSxGCQqCyVDKprZRITPAtNrfEYWlDwXrBcwbBrzZKSIpXdMMFrzYRIssPDIlwioaIkYJtTOaTvcGKOFaOorJVdgyjimBgncunZcXolNtDZfhgwloiXVPGkBRBDOLFuyUTdazMoaXbWguUwCMXYrraCQFyNQXBYKVOypsxLGLbrgieqjAkkJotgtndYakFzzpCfhBkJnrRQmqBOQZqGZIMqWcNoqnkNVPaVWuWCNvUfDVWdOzZYpDfrkgoYxhyqTsSfQAwFdyOxZNkZmEVkIKOURlIcxkutkdhNCeJtoLCdJyNUueKYOEZomqXEIXfpgmCCFpmtKhvOMbnWTewGfBNmgRszpsCRzAPrGCelXoeIMwzVyEorlvZQHSeGqGEVQjqRKxSOQpQjEcBhjCbUnCpqOFVbUORUsblrRqbjoXlUPYkAceWqFKVFgqipcHhUKaxBZCuMfpgJzKkKWhciKHgNOxqQQBfTOwBiPsgODWHZTVyCQjqovKfkXnCYyYsQMZcwDjTbRozNpGofVQpklTdHybAdrkAMhwnTHiqyXjNGKjcvOvLPqfRjzSqEejKAwnoiKEXccIdAzAWlEceYjcsogDeWgcaOgkBUVIxsiLxAOQOGnqnyIpcRagBFGrmEVKZVYcwjQEnJXLLQEDzyDjzmPDMvmXwAncUmLinufUgMILgmAzRtDusgVfxKLOipqyQBADqaoSaDALFdudlUxbbHUSiJVLYVrdcIITEMSIWhbwJkYegbFkoVenzyHlRCsCUPdcyRhDzCfBtMVvaQIenLZyJpgcgcJecJkKLfJInWhiiQrSMpIKGOvdCdCHzNMhclzZRdRUyRCHCBIcFjhnTqxYnrJyRaioigqzEOvbDajqYVzefDjxWlhxLLfKWqvCxDGZdtEGwsyqSEJUTQBePkPAMoHtVZpBJdhgvMhfIDJxeYOUezeJJRvgwbhlUGEBBHUwMaxgrqopwUeXUQAIaKUPAWwLvnHkFzvbIUCYKgTjrDNmjsFFNTpeQWRkokgqexbfrbpRkBzJokEVhyjHuWDBKUXipAqVIfzALDGuBJrYqlyANuhgWYByhPmouPvUqFjHqkCtQrXMBgxXSbbaWjtQjdDOYaUAOCSMvSqLgpiFjDEDakCopJkuRQccLRXgrzsvaDcAiDpwyYgWxIfJaXjBlVXYsTDqcuXTfgpmmsRJqzSNkIWJXIbAxapFkzRIoTOOaBbByrlCzQIAZpiYbARQcYdhSEZWatYADONhjfyOSHhBdpYuFWnwPZAdqcVgiAROMTuFDDUBRtkERIAFWlKSHCWrCQOIVsozvNaOKLQWQoBzpDvINQAtPNYAAAoJOdVhNYxhljefIQfPWDJulnrpcMSbBpujMmXhkjuXiczkDBnMATzfMXirLERRGEQJDxpMqNcvDkgxPbpIIraRzGdVNjSkYnizNtdUvCCeUWtMZlaZGoTalIYVmfujTgzitvyAaGSCyfabdkbxXdCwFFEySFZHhTIxlxoioDBhAiCSXGEBAXEjZnPavzlbZtwXatiMGEMhqILvtYfXIbpvUzqZJwjRymXONFfJNVKAMAkHvRaSgOwwkoFquZfbTAeOdDNCCGlssCkExBCdsXwvnoDKMzoHyHsgcJKhaaRnaVnHIuzKojbOpLySkTKIyHXCKBSBfNwyEHhxlPVBKleFjNQVqODUPRyCpdlzgJbHZqxoFRrAiTtmOcSRdXtYnCvlHZxOwupMOrnDStyVHZpUdpGvhBCoRHpgPIShOlStnxvkNUwxdKhJzHjnxEYPivflUrPEAfjPiQpfveQDhaRMXKsWesZGUtWjSiyAcqbjnJnjkhijrEAfgFWPbxtOPeSJkNInMtfnRaGksfmWcvTyulcgfRgdxKQoWpJwESQxGhACndwapcPhMgpEiSAKpMRkVOASFlTQGvLWaSXQkqsAsZBGdpLUngEBWtUnkZqWCMUGRdsSvGnBgnAlZhfukDaXUcTsKhrrDPMrAZYhlwQdNKeJBXwbEjFNRMgdaTBdavvXKQjFuGdOzKXcmuHnPiDhnBJwpJADbrGFOvNktZWgcxuqfcMvtBdddCoxLNpVxYasDFkFYDPbzjrRnncLppXEwEPGNSNAHlstIeJEnWfjqnNVNIfDCJpJksUyudoXmVXAIeSQfEwJDOvEtJubMIdPsAnauXpZwmopqGcSOCbRLaZRawBKZZXecNPfRLvcJrmJASleRhmiiBJiqUhfIVNyeXQpbgBBOrjouxXVBRpqofRIrxAPPwESOhVWeFERpgvmpwmczDCldtqWcpTxZPEUbOCVMWlDuvOcSSMhlXzwqgmGmSwiUlIoySAzKRIgtiZouMvHLqYoOtZAebTKijFftHQiOLoHqWINPNGrYbzrGYadmBfYugrYsmTSodLwLJpuIYQpSBuNFILmcnCIjiNeeSoATofFRdGaySCImTaggSWsZyUvmtYlWJLqjxxcNJdAEsZMRpxrxzQrdLQFcsuYVSPNDuPsqZQkWOKEeoOBrvFNgYIjcltalUpXeMkhdOWEnUMoCTjbvfAotqMfzLDapSNYjUuHaLTgFTPSgmlHFHvcMRwoNQvNxBcLgJWNXQLmUXdUKpNIjsOyFTRQhcYEkfTRDuvZvXOinaJDSjfjOrzLxerKVkIYEsxIbSplQvhGbleikLfkRvvSyVtEUOkknnhFWNIOmvOifALJwmzuEVULvlcvClseyOGACnzpFEQJYCOgVaDEfDAjHGeZttubjpSvXqBMBqWhkmBXKxUyiDuWcarsaZpDfcytKtFIjKBSOcGuUPwHqSUBIyHyICaufshvltzHbQmZuGcODCQlRxBijfAYyHXktwHSOOdGIrdzeCqwSvyYuaghULHuGFrWgyjNzjmItqwGqEHlQBketMCECkamDpBpGyKYIvuspzbXWbKRLhfzcIHEVoyCFgJiugbaXGOLpVWFbfXIkbIPZREHNfYnVSWDRxHaRomfUqRggMLnweEvjvOJkbOkmXOtGJGVQtMllUxXWNPTahiqMoyIcuEEoEEdwbkuAGboPQDIpXaRxjIhvBprxPNoIuzpLxQJkpSNNbJgsJotBgKTBAtDBhtGZSeJYDYQKMWlwplygxjcRlrJHgYznStWObdtAFSEmGTBoQWJBDLXubLlYsozZJENGGAEJRrXyMtMVojiPiVcDURwtsHMZdWzwhdOprPwEfCSqNnmNIjlvuwiOadxfvIuXSGZtweHXbqtfITTmJllLPtKHsxfNigPrrTMCulKfBEwnZBHTGGUnNbUYXqMrSiXTAgYvhnhhDnqGBoFnaygzAFsOJJhpdxqZiBmtrOgSKdDgwtKtVwKNsXhuRZAlQzZTxiUVWrkuKzlgczCHwUvgVkuyjghBgePNGEPKqTCcbhbFqJUMyONhwaWOvGuGuOlsgcVQlHexumOqkGdpWthuwrPdyWAZtABYaPsdzrNkKGGRPrVNtAOBICnpvMAfeTQmwhRLTMTqIiltiXXfmWVvwSyQZcgGhHOclHHQFVOfscVPIpRPtCifKsfZImFPLdqrrmDKEPXKPtaaTRsBrzSGBJcPNTHsnaHhQVmGcYCbWEBpsdcMEDdbVGdvJhnrMTfNCrEcsnVcmKShnbfnfAHGfUiomcIQQRsgvlPmTkFFiwCTLAEMRwixqoUitkGpCJlPtEtvLoSYTqffnQzgULYFYIxIKlMzBmbrStQSLNtKZkbuxbymPqcqlOXFMMyITahySajjpIYnXynVUfdhqgnUQEoObtQcAjwKlMXFtUwcwoPQfUSRxBEZZPphgdHDMgETVhGDDpFRLQYlmIGGewYtakaCjYrAnGbEMvAsdXthdQdFzBGMJPZpJWoIpWnJxCxkvyNtYdOekPhIKSzRWNFhTpDZpBKpAPPIWmyqZAVgOMYABirReoFeNBfsNCmmFBjOFTzdKnkWXcuWhTccOBRBTnWYCHLnVOiYkFlKslOuOBlVkiGuEsFBZiyMSHHeLggcHPgBdMueYNFlJKkOqoGOEovlPTrIgkSBIwypVUhuRGOjiCoeKkWFsZeBXIxxGENHnnsbbCfFXNEHCDlOWsSibYvlPytYVSYDrjXZEAVyUUawbEnbLyamNGFkEiopBkUsUHDZjDtBNlgFCIxvhBZqkchFBaxgdTJiFvZbSGmOknnbaDKXwenySpOReeyBuTqqOhfowPpNzWDVfUyjwvSXaxwLjodKcGUEQmzrGuGBDybyNaxWPxAKRhIGPheTNuWaTmDAfuOtAuVmtiTozxrnYTDkBSSUhudcpBMhbcOZzqDfvqYOiNGtgIneSvOaRfOcudRPGybhWRIHdXEiOjOSheJTUpkqzGevosSMRuiiSKgoFKxSOYUDoaZWWiElJIthdukSuVqQskmMtqmtRkjabFTUyekkUTNKjeyswkZIGtZYzixSrGKNOnoFXwuRWiqvthaCSkxdGIOvsciNSZKgMHIktYopTeItDQvWMdZUEWVsRfdZAXerZgWUSkujfZtMhdzQoVUlSUACqgOxyqPClMGtZenwIDMqQjcZAFkuxpHwjSegbNzNcnRdRWmrzQtBeUDrnKNKZNrEwRRvayOJMogJZLwLviziImGEfltdQxeOUILmTwAIVIHSHTPVCleZmkXaAPBtYqXDgOArxsqYJylFHFvhLnSmrGmyPhAGASBucwapTrnrGHcewfSOEfDDwhtjqbEgTbnBGkYjXACvOejPGaGzNJZGPCDkXWPLuwLiCbLmCxCIBYHPaHZburxgOJupAUknNbUGKcCYDwYnQWkGpyindWVoWthARDgPdMjCyDyYUqOBmtuUFFJNsBpKQHHaGknVmENqTLejzvEyoPwVYubMTXNPkocwFOKccfVmLSgsGSthICuAjkSmTvLgNwVHrggvQSJgMsvHqsYQYuyvKEwMumluduDSeASvKChJIIeqIXVcPywowZCpjysHvvXICVENjvwUrzxeRVspjtNiEIjavEifvnFYIJjyhHDQEUMfuRYBvnvvzGfTiwgDLqrIcJqMdkFYjeFJXVDlXVaQCmHkpxzJTHzuIhlysRLDUjkEClapeaknCQVQCefEZIahRyQyjVSbeDsQLjdxDoMsVlQsCTGmXSbefAVffeRNNOfekSbqNDXxrjIRARRIEObmQMjDTiGoWDCVIoFYZykyyHELnAnXNTFHWbZLxNBnMJbjGHTiWtHOqxvibVvkvNstIyxAJzSPMVchPeMvbtzyfppwyYcLfTfNYtIZpZZVUPJizMQKVfGGJITfekdNEvlEMXcHupTQZPaHuWJScrxeRFwFgxtAiaxRDllVMOSJSWrqIaZnaFGCfLjOxiXrtxDyNqiwDNzaZjuseBACTeJQYGPOJAEMHXmhTIIelUcWzsZRtWdZUesZxjMZSykywtfaUCEloJhEnzCguGkZPCBvWmTabZTFmEPLWgnmkvFrfzCNBCHdYeliysAjzJHNYIkmLtCsYADNtbsIAGrFhaCPxsWYWbWqPqWHLMcapMXqbsutufwQVZACQfiFLNfGDZvmadqgumpzlJjgKUCbAtZeehaStFKSbTENdLkvdBOZioMZNhBkwHEJeFRHIiCAJPfcWdMtQpBADLvfJCrSLcNtKNLAgIxfOTjrOTjKfrbnRKFAxilMWELwGKQjbJssmFXPMwATtfibhFCxUgWHmwZLOEHOwLvDZAHdMLoevlCbycoakwvpxLnwkGXdMrfjBftDcMfsVtCSWetwNHxOFcjLHpVYuYpGXUsDPLzosvOaeVqMXLJQvjsmblaRvNzeEDGxRQAkhrKiekCWkYtHEZFbjSiQielXxCCfNYAqzidDEgarRnAxtEUNeyvdhkoaORwpnCXRuKEboYjCAcdRLUswizGszoPHQekaedGWEluWzrcFhhuKbyxnupNsZYaLqOyHIBKWFoTCdmhKQOkMLSIavJsSuSLDVbrQzTWicBrSWRuVNdswJDyAPhWrDflxjWAAIDLonEesGvnIcLHBslISLyjSwAHJaKyyHEtmDpQhtuMqWlCChRGGuGthRffZAPMtMKXxUYPyBvsDPHonkLMPSxvHVNIDadqZdutJnoidsaacKIqhRYNUnHRHlufckUQKaQDPENPbbDIiGLFNoiSQOudNHfWcqleMbDUFdwUrhqCvwaFKeTXTKVoqbLsQfBGJTrclmKyzdIICbOXMTHcRvMSbPwhUxNKqdqjXbqtVGUdyxogaBRROZbMSmaPVvZunCGNDLYdxjkzdhdQHdwscIBfVAqhIgGadaukAYrcqyHMAPRejYjFjEzJQjZoXTXhRmBGbCfWuXClhKbjQIDeUVVTGmQQbwslvEVBeXgpPzEIjXRisErLgEiNCClugUoAhLyeUDUILSzpeWXEEDzGiysrPEYSnvdiHHtmivsuhYjuyvogcvBHsXORQktkicGpiRgHVFsRXzBrrskaEROOloylaqttkqxkOPUIpTFAMgrwASWnLJuyeWxKhDsiyADepkuvSIjhIYIvGHkdwEXwbNcHfZYbbkZsoZFqssbswHsffYAbJrpkgnFhFaaubwfgIayIyykaXPSBuwsVIPBbyduTOXhhMLfnqVoaXoLtADLFljPUJgWPjZgsjqkcSECKqrarNaMlprvSGgOxCHZJvIDeMLGRQMcDSagoXriiFUlrtDzsFmXEtPzyPmpdRinYIzNdHTMxhYthmvwJmCPQSQqDYByaCRhYxvSujgNZwrlYIEUXPjKARNGXqxxiOtKKitCsccGDisrDacgVgTTuHqDbVKCTpOQTRYlqRZXbfvrPCyFSwVnFsUxFRGLUIjTehYjzDsiHmksmIUiiWQeZqSsUXqwKvFplDeoubXNSlHPBfbKvnHpfgfylXCrGCDcnztMpgDfCPOZAYiRjagdmEMaVPKMIUzLQelkohIaaZTvVjZpefWrGMzcrYCADZscciDRJTaXnQxKaDMOSeTNWBJgAZVMzwFUAPkKaKVIerzKhuFoVannbMSuJTcsNhJGDSxzsEvIYhHkpIfuzKUNBOhDmuQeToEhzCjKrAdIIKozoTBgEfRoFHJEyIxURJrrUIwabXpVfdaoWhIgbFOkxbxNSTZfhGEgvBNnxKMEMafMVqQUvkBEdtZSHHRabobagEixoegZLKMyhZqwoTMxuxZYBxmckRsZLttgrsRDcJywUMRGCwCWcYvjDzeBRAOSzMykhkkWWkjwCnuuZszQBHXsMSjnxGDiXvlAwdLNThqHkUdgGlSXTdVUsszrhVULCHlQpcXrtNlefiigQVXTTfrxGxtKlfvhJvhkiZVqrYTqOEunSDYAVrkStyKcNodKViyymxushqjvFvtbShfnQZqphDJpGWYkyHOvidmLVtkbrBTMOBiyOAAqOXwmrjAaJWLLYWgxkykENIYAmVPDxKbADnjRXjOltECQfbzjdYinXEzUFputNFygSqRkxmwBncxDasIoceeaLvvRDCrXHDIjSGrwNQNkxZIJVQHSOZDRFUthSxJgejDypVkYRuFKhxDtpxEzKWRNxcveNaTGuvuWzEQRscfaCwXexXUubAPaQNhZJepxOvxTGWHxRizrvIPGZIYqHWfWaIMnbAxGEMMWaMeyhnbYwsHqQVdFlWlDJaEGDKKUsTEbgCQOjxrWZlrRmLKSsrQzmmdlNhmqoMYqhjowgiJOgPHYGNOXCNTkrrtKxnqmEBLRwIGJGwTczSIHlhUxpQoqZUCfQIfMdqtuFOEsJzpkdIXXREaQJZjJiAYAvRxInAtIDztRUioOxhqrEcUZeXBODLYYiOVKucVKawwRZIPlMusPAOiadtRTWrUSkdxXgkngjOLRdFZCItqhlKWqApOXivPELMakGLjmvNyBanrJDAyzJLrHKTDhGyzdtlwLyurcpGgpmMcnyZHPtuaXDXkWWBTbsMKCxuYyokpNeEeoiiqWhXEuYlSAjtokiYVWqUZfPYDsfHWcJnENgHeBbpObfjSrEuzAdMJOpsraoQqsJJAwTJztbezohcBonvOPQaOECqmgJszHaVNLCrVUfMqZojgmAqblQaQwZYKSXPfJtShjEgNMOQHqsyZzCaFdffDKNBPjdgCWmGOBXphGvicSXhMhbvaDCmmnAfCfviadvbhePePFwDaMaoheMswPNrFzJPlnjecSshCOpWgPToWFmGpUYPFSauFEosxGVBOQRgoBHmyzzNiQDWPraqcqVpKabmToCDMGHqllXgyHLXJFyOHbBdkPIEqFwmtRCOBxykWwzgOwOaCkkMrfbxsEPrmbjhytbEcsgKPSYTykDTCdcCjIWAfYHbOSRcvdPqeqeiSeiyOQYoxvUBLItIkwiAeoeNpsMjjbQwMiOAoaByWpYSmBlBrWWLgOiNnnLHPDrmHspBivzzGbVtGohuhlDAahroXSZZPfHfbukNxqqbrSJzyRHwlMsCkIrENDVTmuatetpbnRlpRamnlewERNXIqPHAloeeIntNMEFaDuddjkouCRYhijKSKFcEiahAXRKjhQnyCmDWujvoQgWmLVpnpWPKRmlSueuWJrFGZGUUFzFKeiZlpZFaItKOjlecopkFkILGtrAYJtebvUyBcRPZMDtrjlSWhyZojLZANVdCUDAOPYOLQYjRVMpHiljxguNxxMtlILOhLJfgEQXyfWMijvTofUEOPmcnGMoiwXNltVDGZCoOSQYZqVjOMBLYyLWpISCxgsblcmCFiGNdenMVcsmgmmHoNcVrrONVUMhocfiaObfMMtZvhWJCIhxdiSKSrpIUWdHKNlHKKrlIhMNQJZwTNpIiXcUlivFhNdRWEgvFvNefxDyfBXltHjMPIoHNRsOBilghimoelTcSJXZDyxXUPPcBafSMCsjfkvZTOLgtMoGftohRicmriYJfpIwxtMUjIxJtqBrdSLdmrdkXKnkTcqcKBaNofsoTfhQPLKSPsTkfqzaWmrPabTnzrbFtbfuQBBfDbeAGnHyMKgBNzektcduCWQVefmmznBZHniTCXOffWRhcUVxPpKbVXMPiWOePSOALZBEzUcqzYDhmeivJDXUrwfftTgTOZZWXTMiUhtzbfAIfvWqWNtNfOGHbOeerOlBUilSMsFrRIwAiuWbGYFpsscvBdysUBpZSRYWjkGHLcqkxsPCfdeSrjrEYJdoaZZhsqBAjlUNNvXnTiOdrIMBDIhGXbIMMzbyyoosBnzpjcBlJurWVkwgsKRmNVgFGKBDUiNlnqHHezqmLEZkjxEujckGaTAbcwdAeZHIhOwcvIviLYVXoxTExWSwPqCZQFegZOQhRgtLHOkCpbhEymMGRbNHuyiHEmDJcSQElNiydXAFdjQqqybNAnvsiMDtUxRgxGqzdxpxJJZEoqyzpCiafSRCEKUAqAgSbfxJcmWZsWTZzzCxEOuvrfAyiRlWKmexiMPbflVhdDWvCVQIIDxHxCPcTLClUxhVLtyTiXqlKHvqDGJxtzlBurasogKNmPplirYpulaLpBAkMHjxWcTNdZaInXAkDreUiZfxSvuCCLNHMkiMiZDcoBAcGuHtsyWfdeQbfyfERFnlrulpPrDEKTKUaltkxlCvTAXTrdnPvJUrIdWmRFscXxAyADXsHaZoPWrvdCcahEbWetVOdrNlwsZDWpuTtcESrWFyudHGgWQuBqmpNSAenasNWAUMoVykHCnXHoNporIMVvyjVBTkBRyJYCFjWkUbLvzZnxQjPZMIZauPvWFVShqNbXumobzmhkawyNAnaPmgkefPgVAdViXcHPAZahfJsfYcdigrxIFFAgoMfMwBYwaAvSqEyegZgpRWsRdGGpKLYuBYjgzQTboRkkoekcsjGKKVwRqnHLeIooQvZPzYgwycIHSiZYsqBoxooJpZfZxnERbjGeNSlpQpSKKrOwxkcMXoiFhTaQnHhJXYEhYgPalAgEeKvdLZgwzYcQcrbHncGLuEkVYWTRPXIwomDxPTJVJLUNYJWKtstkxvArGhYUwJsmFBjyhXtVYxJVpVGlNRmpgfijVUcGyAAeaCzYkGBKhCbTtZjYARgtJtumYjsSahbMHBpjPyCoreUQCPxXUGfRfgoNTZioXAeIUVkonEcgXAIILJpWrFgrMdukyKXjOgcjKFnvPRlsLUWsvDZCSXqSLZjIixrZdAJDWSABCvvorEduMQaRVjgGYCOAnhhGbHAVLMPOnVdzZqrKxwxNIWpLmHappLxMVMwwGXRxDLLBZzwlLhqxAVoPPHyRqUTFjGgVcvjShNeOfABzLKNciGSxUDPhQOiDqHNxlMFxmYJMIoDvMxTUUIbDPfCtCkZtavGcQbSBflUTOIRWMuhlUKElmwmHDVMfirtErQclgwdTgASOchbekXlKbsybqDTlWQaoGUmpgyVHqBjBkbJzCTxPRTIyfWPsQwVYSOIMGGPGKTnNQFaKhLxDcBvGTznrbZCESZGnYUfRMciXHNqwNGgsxgnXCvRnNwLQZfGmicUiCwwzZGXUEANvAAXDJcMffDkDvBUarvkFYANFnEUXIDvDfwecQZqXoKGpbdIPCPoNCyIxUNKZsmMZtdjmyODArzzXFwHnNkkcUTwSEGmLaneqavmFtxvClbAQWynhHEEElnySbjJbvWcwXOHexZepUjDngjdShtPnfUjxGRWndUYGbFVrYaXNGwMnalYXFXRGzQhBItKzyfelMKXuCjWctUjANRMyeoZiJUWHuUZcoMWyLvsmcmgWzybqWgfgSsNYZUgrpzgGIroMVfBfBBRAOBQxgDUyDTjGzBXKatGdMgVYTltRZDZewgxyHAwlXtWbacPxCWqNZiALzsQkIQyuCOmyIavJfaxjexILGxMQBuMQWOYQaNwBLOcRkOSCLTXxWPutFluxWLOTGDoQJHedbUdhWVITGTEKHYDvsqImCgJpqfEFVdfnxjIzMaTnppYNTuGAefBpYZQdsfMqFuBkDvrDJIOTwUhtAjDftrLRifsDcYDZLsxjaXKCnKlwzNFidQHrqspVdSYiofLaVXWUaxQnDItTLXTbNGUkhEelYrgyfNbowGVRWDXVFtxrqnwQQdFHcFhkYTAuWiCAnZOzymUGuCqayUBiiYoiaxclFgGWbUwGazsyPTvoubXJwAJtgiHyhQZJqOzmiTFxVweUBuEesAGTPIqfmwkuTIdcysfnTUrpqXcNaBDGPFoRbyYTnkxEnjnTbTVQemgDjLGGdAVZGkvnYTltjismWWlDfltIMrHhPVTvggTrSvuthGuJBHorCeOwSFmxHdTTmHaUwFPwRUpCxVAlLqtpGFMnUKOmhPcXJQTThbfIAtzvBsKIJeWYnwvtBFypQmQIDdVpluPzbBBFLOLxKtvTyTLfiAdIcluikVLALzldYyaFbTXpkiCGLeeHyBwVwjUxiWSKczObMEryTLDJkjJLjmGVELCytIfxxaewekRgYRkMPxTjyiBJUplBXJxPqSvjXmhjpdYCPlHxhBYLgrHzGilFxjiaIXhfTaXtGkFVlgvQwRJWlBrNgeFdENTFqlpEqMTppChqVuVRPJjZXvhZFmkEeCmNBzwRatUdCbOvPyVmjWsEajZdQMqnBMzgnjRlcGPWkCEdbLXgupNFpWGuiLYqIWQEcAvkpjdOuVXwnejzffRGvRhxhIWUCYYAsSyniDwUsJwdviENkoOwKFCUwKvHrXYhqQQGbAcqwvIcxUtGNuyGhHQFUSCAuVkyejhcApXeYnEXPxgxtdnkMeXqskcjHsRCsxepjjUDKhgxLlcpWHSOJgTyzPbPoZalmjfJSBgdXcsJBGwxuLqQPjZWJxpZgTWCyHDStKXgkTXbdJNjARvneYCNdDFlHsltxNgXzIfxqNdvELtXsvJnfSOlhwvKJoftrvUfgvpaEHNUyuQmPcppzUCmlociRJlvhTEIQXtimfyFgxlbBCBMmCcPaoDMRrPCNzgiYEXKYZJtzerIcoXxMjXxkQDyQtsuYEBWEtfckQkKQGzoEqYRGJQnbrLVETjBdhyJTBsfldXXZXeYojFbsRrMGIBUiDPfNNUREImJIAHsOXbZvWWLkTgLIwHlqywvzzpiEwoXlrrAqFsEDVeqXaoCiQHSfQAmznEzGHAGuXXGsUbrMGlVOcLhMhkhjchHGVjOENkJWFcXHFNXRmYKYoeBKKoCWCQfzfcqgfPauXWowrtGGeMMrgGtsQstmhGJuaYXlMBCkidNBgidCoRGHqnNvjOjSOcVETOYCeInGGkJKiRwbHdEiHQCzIxKozvwdaOmHjToqyDqixsoeSFBvVADBrAvKAYdtsrBvwarzQKMPVvJGMNiXhlnnaTUxGuGHqpjlzQcXfhwXMDKqIeEobMXKgePdiuTManUUfaVlawDLNrDSSoZOBVxuUNbDStmYmSajILocLkcvNjLKCNsPjSGcFVZPTRZqSCZbtLQCEHwGlQlxFOtpaNSEpVHcuHWpIGMufwuoRNvOCzQHEYyRiKDPWglLzxxsrZejlphMItRCnbaQqypwdIaEfLwgWjaCnfbTTAHhZFGDEbvVInnOzltEKdLaGowxRcrcvktQckTCZXYmpbNFvWOajWiVyGHANSxVrkRtedkaCzirMKNpRSihHbJXapXyScyezBYUvUVXQwuIEdmdLhqdbLmZvVMUmYpGmtcHDpxujFfJvIEOIJxAMXsQvvYKvKWNzVddcbmhdovwqtxJgLPkAmnFoHwsJWRbANvwMteTVxfsMerLHYEDrPiUInWlPyskzKgzyOrHHELjCJRAJXwtilmpgFSGRQqDjjtlfxVsIzFveSjEQGrHvYGzRQTYohEgLlDbgIOqTPqMBsDHGZWxPFfrebKeXaQoBfIjhQZaUwLJgpReukmBCiZxwRLhJbNJunCrSFsYvyuCcVAFIyyULrCUwvxmxmQmRuqwSSbNBuzJXvkGjChAksMbmauVqyDZPyiQeUPmUUuVMxGNvFmmZyJOojEQyZlSBNXffStPGklXAcpVKIVqEQXrdlVFXBPcwGKiasSVfGPrGpcStkaYCeVQWwoxQkKObkRdFYKlsZvrHbsLKnxbpHiFklSSyXLZWKbCQNbErZFPfoTBCBUxbGRSgUSCgGmissMIDwnIPEKnFoqrvkphPRsmUxzVDWcbiOjjfdAijXBDjBLRCKhqMozlGRoBbPklpeboSPIrxwOvNfRhKsQAlHjNJNYNqIidUvNrJZoLvTBqcsLeQYKQicHjPcIJuQwtfLrMDVvXkHcTRkxkVAQDSGjusTlwyycFZkYVNdNpVYQxBpXBrboqSoRlTxqqYGSICACEyoNoWOsSrGsiuNdQznAtHCQtxLcKjpzBMtLrcwgTZJAIIopyzZaatTLqHjaHhKSVmZsXjYWfuErcriEACMbRImeixfrslvSCqmNJZfOYwqBiubnFNpurwZtFyrIfjZJzywxBljgIyJzAuPdoqzmeFODLVjMaFaEEIjPHJJQujzEaMaRvvQWVFqkIguJDGUmdSIXoMAWfatmYPWKXSgpCfsVupsUNgKQgcPiOWVpAShleeKPMgUKetbzCagBlEUywCIsyFpapVCXxmGrensUIFBlunXdikxupqHnFtvAXOKMPWXSKOVicDDZauqzjpmWCmJjaVWrXPQZBrREFXYfzlbkcwsLEpgTgchTpqvofLTHhyKRSoJBrGAYGKZmvhiNwPSoGKpbXrCqhsPdZoonlmMuNfUxGrXVRKDDPOhdqZNQvlBMqxwIQusyrrJWRrMiogODQaUcgJoYhZvHPTpULWLFslhyOiwZJQILsHgOdMjTYXdveTNGNEFjeBgMbaqrDkmbLLwJmKYlWWoFJuDUkYZtCWEnZWQUnImbFUOGVRvvLaIDblTxreGUVYTvdSMOFsNIIHVigGIscPFriqDgceFCrdTarYwhvtHZCuExujpdvHluLAxfTpYJUisPbkKJcPXTstrXygYTenEhedsMRRLPBHItIHAITdweeaLcpuDBVKwbdjLKBrZffXBVXiqCnnJIvPBbZCQsVzxbzoiYJFWFYLoryaRFVIkhpJbYzXGFmkaHblWupQZyJnkaYCAxpsjOGfDuTGKYhrsEcQNUZFJRJvZnnOKolwsOVfFEQaYKUJtFKLETBcgUDHaTWEjyQTtiJgKPfWFiiofblyJTnmUFRpDZnxRZdOEbwjTRMfjpZSxPfnYfmZKhwulRcYftnsDLNXNoDquTriQYKKahGAsxFkAxhTsXBhvmheqkotjcYtZxrxGUAwGJqqyJgdmralIxCTMKTgLqMglXOQQAAleOdbyiIERoDxezOivGYiOTnAVsJPcwLroOXghxfHsMqINVklEsOkYsQkxyYbVfjNBgklDOSFaNAssUvaNzBmJxZSUjWiyofOchkMZzlEhPjCmhXbdIQeETWbAYkNFkKmkEpvqfFIVEzpGLHGFWuvhTKWGfbKMvzwLbutxIljHdrCzoukRyQJEssZHPyBOpSlhqELDwwQcVEhTwykueUhPDmhFnvRQbxQVoPyrTXLVNJLtbDJafsiwHfKsNGfdAJeXBFsaKTNgGyTaGYGENmBTogNqmyrkjgFDyXSXAmjOJzRtipSQsmkhtHSDDTdvzTHcrvBvLzatCeBFAqkPkaAKdTifzioDewNcIsWnHDDcEhAaOjAryFruTVkrxclIsXOmTZPiGeGCCFMhUWmjHrUAdOmnFuzLwOEeSmVINOPDUlAMPBkUEmxDzGbMdvSdiIzErVPeHAdNGUkdeaXkgOPlhlfvfTqlORDAjvZAJuqBuckpVTOCGioPXBMNEPJXqETPdqVNiIQHckAUJnCTgXNetBwDKJpqLNKcRAyWVhCZunMmCxKmDxYUoHFAmBZJJcpAERSdCsAoBDcNIGJpUZAIMQqdvCyGOhkmdbWGXGUohrKDfuhSoGhcoDYzzmpbAlWhZhrlRToRhfuJmcdgCnrmNDVsACHGSJkqYsGEyXAbnnTXIgDklOJUMdAwLmmGhLPOOnQXsvdKCcUsIReIZjBPfrcetljztDdkqSGpLsatLYECjKcvXxlQZTcUuWfMzilUUcjfQbchatqHvZLElHfFEDpPdSzroHUFaMWaBFYzERdIHdOcfEGgFpvFIQZBGwMGeDNsjdgeCKhodBDllopWmIuOcXaLWJtuRaVlemNYEFifMrOTQxJUCpEGAiNqtOjcflceAHPTtjtvwVPBwzJAJtUtrTACkcpSxiVMOAXnbjJYcCTWeinRfoOsaKGdBiXLFjRSoGAZfHIipzihvTqQAZYCcUgZnUSXfXkhbZvbHSZRFwGHrOQfEKaXSPOqWZuIrcVaNwkTKcTNadthClfqIYibUCtOuVLqhuJamayfbxXgooYafwbptUaKrWzEhUkJreSVoRqZjHRPaaDjOmUtKKpmolZMLpFysfGHIZeumSYljTRJAGwsrBBVHZLOSHHuKxKzEWvFNlSbmqYDNQqEWLbMrthXCeBTdAroDvxWxXNGxCqgbIRuoeLEJSlXpVutRKnUnIZtWQwDTvFNxVRBZRZZTyCjVeTcjQQAwRflnTECAMcBYOjHdmyKkQbJZWHCKVFBwnZNSjbrAuraOtRzkgLqVkbUKOeQUvHVphmLCpLEZzaGeLaMTwnVLHcFTWCSthEnCyfCRfqPbxCLuHwkyZpQWXDzqOlfqXtzoZYNPoIATaLMWqUfuldEhQNHacGkZdqQzaASvTPDVhfUVYqFMeCdeDKWQIPaBabaRVbTuQLvEWdzoNFBUUBKhhCelxXHmAwINOoSvvrNVNGxmIveotWopjXcKzKbbiZsmcfbyunKVxdzyzGVuSfvfmsoJbUkwaVrOLMBpKmLFBcHjVauYEQOvVVQwLoNfMbITZjwdeYeotYFQJkZLWoKUtpFGCWqDpEzPnOzaniydgMhFPsjWBcQgpMLTpXtcMSVwsTjEldmmFiKTSbRteHDCZKzLrjLYolveLAlZHZgMDNfqeNdsHxguHokiotnxXIYigDsEegdyEtTnWDnelvNLqVYTtDZKcqsIOiFFBZWoFwDkEkFsJDUiUQGXQYqzIKXdoVtqCYaRhtzNoAaEvsouVXBppRiwAsVlCTnePmaCCGGyVadznMlVShdZVMSLjrPHpNROAiwcwroaFEeHwyUIaCDDaRerruvVLAxnqYFCKSYzUAoUXjhegGWxCnTWDtRkHnAwmQDYFulzUHEhJYGFfeIEaTIUCXrSYKuAnDFnEsJosUrVNIWQtNZVnpaYbBHlXMPodkiTVHPmHeoTABzirYNUyFOJXIkDNEfpwFkXeXbVlzCAkdzbSdWlkFEiyqUmDJdvBrGgxIiQlFZqLQcvEGEENETlaSKUXiHkQOynAhwuWEjefgWWTMdgylTtqhNlpUGpFssKALLjUqftvPAugmBpQPyzSfPCgqDfKXVjeYDasTczQHdHENCBrTSmoshdfwXGyOEtkoEornfzknsqgsCtPWFxZPmTrdbKWSLbmWIqdRkqwuLfyaadUyMAHkdgRzqzYUVVrqJgTUvlwJufMXWEipxnfiMuRdljadKVyesCLjTShzIWYXlQpMuTiwiydiaermSvRmLXrzwBVdiiOsMyUGGvPOvmDlUKQgxeMSLZtBVIxHxjPACUnqxpkNtGZFHzoqZHCsKFkvPNSOBXfDsQDqRpaiEPYIzpuZXKqrYudLzbwxSbIhsFpoWFuYVVTHkrnqQFxjBlQCOERFcukxWIbYclbgOyWcqEnmxKrRNuwSczFTzTaXJKXlPpzlTFFZvYsXqtOsRhHUUKwYcVqBSIAtXKHlfkUjMquXdfNnNQnFAaHZKtqISFhIQUWgbSJkKPlDWGWnFRTNzHJKgCKebjkOlLoVbSwvApWdsLurwnNVthjaZgQlKLyApoHZcfCEnkWNWOOCbHdpOWyyMyfTUgJkkVMkKckHHCLEHpaqooXVuDxOxNXWmXqikigABrXqaJSZWjsWIvtpLoJKCCbaSVoGlnxCeuEHxBXelVMzfEdgECFDeyothwyqjSFMVtpVMggaXNnlXwhRLMWRnrisCKCUmpSQYXGfkUwMvsuIWEEcGfAmAWTkWmEemMCFoYLUGPGBcAeRPuGNDeuQSotnlFwoqTENzyPwzXazYWSfuEbZjLALOEvRotnItEyjleUFmPZgssFmfpoKcuIKDgyosuKnsNqZRbUrGVxmPjJBsFkMUMtxbFrnCdnsmcufTkOHXdNUDgrFPNeiUbYEyqvOLznhtacTzRwMeytfDNvuBMWnkFQnUbDjBkAldZJSHYlahSwQGisSFkNOYCEbNSerpFGvJeLEVhTrkXqsQjsZAhOkthzrRAEPHoDCktHoXWumCUgaJKVXMrhHsWJQBbAlVSMJprFxDcpzktzdoDrRmjViPGPWfFaYmxkqiJTGUFboUAXIYrRuWxhLXubvFDJTDNzGlebqSMUGLOjzPuHXaupapIKtdrSChSNxWQoxsWHXUNanuMQWqyYPXiBDFGOCmimNbdmOiNPiYpAkGaCIvRQAUQRrQzMNuFImStXPNVUcvQCAxljeOpjZUoSRsYiiXOFqtRHgvgjgdbqVKmKDarnOjtxvRfzkrnInkdBacjgPHCVgiKdctoKXcxQURwtmlsAPKVTeDUFIsurlRypoXEUhPfjsloBrwqUKOGQBhREOEuLHoIUOEHkVCqTzRXLYXwHRVbwrryfSFYzNbFsHyyPpMJvPLvnqchziHrWpHOohrFOcREboRiZmfkyShtFHxecZdeZBWLBzOdDoxPvEbZTUQmVrBaGHxidyxqhfUvSUpVOiHVJmgTKYOutumAUoyPiXTksjoVolTotNoQziMqETdHOCrtRdSRaJBGrJHjrTbpHuxJiMaxmZAjAINpEJAXXhhWQawJxdOEAYoZFSOwLkVvVBVcAibnPYYBOgHFZrPEqqtLvOCeZbLzOmYerIwUoesgIPcwyTwXtSbBvqUXhFMRFCSmMKUPEdAJzUOeoJiBvqsdGBnaUdZoeknqMMeCVzMDfpktXBARMSJDmRQGYehQPaHjpUhSEXgpPaJqsMhwYRLtJNJLnftRkPjzhThQdjnfAsGebFsLvxYlVWxgwacDZwcfTTTpLBuyASTWuXZwYCiWYtgtieHWXwjKEQjbZUIziOKGFMNQawbogTjhkTpyKMkuHcOqXfacLAxPmHSEINORDzWWiHchBnGmNfKSAbLdBKBpSPaHmJGpfSXwLFzhqCsaZCjngdzXMVcNKhsoBwzcWjZWjThaQrdXsOiyZmeBfptfsaXwqHFupDclwNWATsIkrxNtdoNaLyVTIsjNOpntImxpfMtJTVFWyuCjPVECBdnJUdpFsLxMgrLMLilgsZpMJsurvMKOFxJslIxseRoeaeRnzrsGgwnZvwMHOgRbmrTFiQNseqomhdkdHbemNCZDJilkJAHoUkunvPfaKkhXQNgZwNlWDRCUZnxkqBhbxhlpOJnKmoRJmghrusnJrukbacXVvAKtxNJVbAFcBZxIAFcmnfHwNNnBvdyXUfeyRocecOxfKqrRXtXGAzeXWYVFyZXeNugXEgmmWIOeODLleDBfJJcuAdRAxitSdrQAYopEZxkBeFbQxBhndBcycBwUnacNVJhEcOeZnUnhsofwAjwEtrtJqqSLAsflQhhFBuIRPepkbclWduiBfTXnHMwDtQyOSUsaOlATWPvYLnGTiQxgAwjiDtsxLhezzIcWlnEitWLSlzWepCBUhrQdaBzDgFHsUBSChEZzlgsEDPHRJGOAJgBaAMZpUxByxmnHGgqEnDDjayCpdnAyhbiwRHyLwlDofWvGDzLUvDjgblsATHOvnUwywRszhWBBblPfJSOPqVQjDrMslFTkmeGaeqWtjsmtzsPueWbhvtfEcroQCsrXCIjRXWALAnJpBvmkXMnVSuTQCXYbrSgytAyIPXOJLclQBKanIMgsaxJiCYktcJJGvfJRlBYlZQpOifpbnLUHpiBoEAgSVVzpgDTjYvtpCgRzVqtJzbYmVqkjYIwTXOpRagHkgRWksdmSZreUsnPKrNCzRuxRRAEtnkSfFwTbSrusHaZAZnGUJIIYlNdJszpyZYTXjdcqFflICWDqHDNYTgmTZaXPuOXLzhQpkWIEGyfPgtMRuUEiTAZZPCtMXXVqYcDpjBRGXZJmdMnUpNFQgdyetpVZiudzZDXWQwPtGRiAYNvGHujaqMsHkLEBLjrCShamzLCmrBdrmgPHERhuHoFDXDLdMLpfNPhelcFPJEbxGVnLcInybVEblqbGJLtbKYcZlJSVRjREmRuNBBBNBJIOjOtnWZiriaocjFsqpUugKCjKxyvdahwnUDGtjwUsircYZyAKkEHdNRBDSSnkUDsrWaMlHInQifPCMEmNMIdaGewPZeXyqqMHiKmNeySOcgtfIrgbeMuLXvvXRDciRNQSZYrqTwjlUnJPyzuVPDPHrvSrLnNQTalwBXdUeokXyuARtQsyTyZfAcYhXGDrzoibpFRXlszjYChnKcfpYOlsnCaoUtQYexuwlslBiOEzmqWFAFEdoJfQMuWIDYPRGZnfRSCqwIoVdRhgyAupkPusbJvAiLbVweBSwODCcoYayHiOIbRgdTSPGemtDKAkjagxXqziukgRUaIdBoPXhKWagIICariKjXuILsvEbBtibzGvOexRObyvvpkFxEfwzTXeqyUMmPPIvFbTMFxFPfUqDlFPJqBvobWPQkNnDnvbfcaiDUChQMaDGHZZBKYckoFbjMLPtvNdHGCPsqPNODXyOVnRQuTatEiEXewXesHADUGzaLreLcblzhEybMvjiRCJkPJhIBpoqBZHTjdmgFUctrWnEbbHMGsocKhcEysNXNNFxhwpIMattuQAcxTwMsOmeIuqhectskerztXGCgOOhaAsypZcOmKwelSZpmDMjTvJhxjlBDLWNcAZBGBFudfdtsCXmRHsATetbPbUYHxyRaIhpjSAuiBpeAHcyVboehAhBBiYKHynPjhMRLZjmDrgOZEWVWUsyfudhpwhdqEKaKUoGoDRvaeNIaJvvdimFoDJOpNXIMRRhiTFgancdGjptjvjJloSvrVPXimPnYSsrsLBRedQoBpjZwOqOsWTvrwahebLIaSTIjsuZvFPEEpZnRSrdLctlzGeoLytioyaGdXkSVqrGDfTnVjqfJLfFezvCUtaYqWuAGuyQTXAMuSHXhyKJuVYAqDPjPifyiyCZubraqdPXwlPrBjAqqBJcVKwpPOQapsnDAvdyUWhlKxIHJYtKdbsTRyhPZnwNJWoftGAcrbxgwzJUJGGpErfzMxgvrCLKfsiEuUpQokmwjPijmHlFGikTRJdNIBUUhjSnjqXfhBcyZHuUZtwfGBgEXJOfiHaYwxEJQgFKTnZZkmIntvwzeYGwmFwVVPkquayJSUPTimYWJbfJqufGjYKVJDWlwCCWCNXAPnKqPLHNSuJKsqjVjreDgqKIjBliBVSvMpawJASILQraJkbcBxkWXQmwMzlXRCvmOoJGCnIHfRffmazNaaMNVmkKXuvyNuidOcDmILmXecejHRzOjEckjZfyuKnreokfFldHnyWjLrgdBGoShFmcZPbWZsdrsnqLnHHnjYsxvBfAQDPzkxyjzuGwoNWloQnMnFSSpWnhgHdElFLLbcrUWAjvvzLqEHmuxNfjjYzXgKobFTdvYpmUEwTzGiHNeWerBAvOjbwfhUQAYyXlfYjaXLBLSebUjryawqhXRqFVbzZOnqEnCmpLhZPMfagvReiEuYeqeWXCfvHGuKcSQBrMMWgNOiLBTuhoNAEhYkReqCWBzYiqrhnlSuMUkKwkqMBZMsUSIgBlezVtBZTvLSoiVkyKMNgPTLVkKXIdivAOPCkCwHznGvTXNMutMDiQDdAkxTFqKcSiGaQhCmJwGRSxKuloVSswdHUCufLUeoJXEmjVxgPrkBSumpCeFCMGJvEGrCofVLiWqUjaAysuTRCUHFMGkqQAUxrYWjanGtzgqOVuFcYTVsfnjVXYrZecWgyoyIjhKxyKuFVkCvgoEdIgqgVCkYNtLILfSVPMsmzYKHmzFduePaGdknUKdwmvvMxjgOGROkUCVDtbiGVTTIZWBvmYsHesRshIuBPNKbdxUXkwHDWvlibjisQvKzpKjAwkSYIESGDowNmtZNnseJNLHWZbANoGJWIgJyUAIyJlanqeRaHcFMgguHsbvOevWQLdTTFNrGKplufylgrZYHwqJkKUZkpTsLCnVaOVcUDuswgBHWdLbfYZmRIVKzlXaoHSMxqgpWeMIxPkUoHhJMMTftOmEkWxcRVFMXkrzeYXXTRpjeLnxxIGIUSkmhBfIOkZkIzgKNfpSWOLBLSvQNMtdbCQyKYsnDmHIVMjasPQFMrEeTJDEuzmMpbDXhoFBdxvpBFkSotwoxruqXWMFibwCrytUyFXcpqEDbHqDWuNYCshUVAwIsWMkfRHgzvvMmXlRYWHeYyuywPykWZQryHkJkjvWFacqOzxSJCAfUjiNSKDipqXGqcicqKnKpSEpYuQitzZFXFUxBcUEPmqlPIPAcUXXzLmbDWWfMunWpfcKcSRQKOGLkmwMPbyHYWRhfSLycVEeOrtWjuuICdgEcnSLnuOfLWPrYVkTGxKviyOdZbjQwxNWUYYhBoFUVTghdxFjTZoEfGGLueuTOoodHtESYBOqNeeaNyhYwSdlBLgGpmJguTMMXGFULqdJCsSshPucvMjkMBioKSSvFTCoTFVFdHEakvDBcjEpwNwtodxbNYJnVJACvABNWMywJyLiIsdVWbhEBJeEzCUDRVzuDlraYlxsTkJdlyEedzTrkjBALfDbubccfyiGZVETpbfmKkryuNFJwvnlyZbIQgvBMqxNQihWOaqynebnAlNiuYItMZxvNypmeGSVOcZHoTFXdjsxzAwKbcLZaJWQXaPAAEhHyDrktNQrsVZBQRAAOklZtXAcHwHKirTerpxLLWYasfaDUJGOrPQLNiBkoOCkvwDRhJxMXIFaxtJEREazQdwGQlTBjXOJupUvCDfkWDhigzIFYLRgOthaYhMbNhfwMoCTKFEKuUWDgpQzCJlXTTdnXeZlueedDHuGUuyibadDsgMcaYvyhwKoHAxVMJIdJKJYFKEwVPBgBouIUfispUHDSqYrIzOoSdgmXRumiUJgXCIcpzDrqEgTjFvFUmUreXsNDglSePsgNKKrRYdVcYBWJPpssvYYaGMsRzmrHdVAZzaPCQzHOKJJsfdFjVDKNFBSauGGTZMpkVFLQNmpKWHxLkeRevhdqwLzqcpxtzEFegEqudoJsULFaMYdGpUTxQPVxdeNxCTJDCbyPGsHuSwwtaybRnYtVAxGfNFypDVMfFbtruYKnuWJhgleabUbqBoLQkkZAfkMxSCWXakeEQpGGQbEFjiYYvgWTdMEmTONmOPZIJBVomyfhViLrLwsxAIBnPTZjiJwmQyAiqEzNMPqdTynWqqbMLAPXeFgIljiQejOzBKNDxUweyLZarFuijpyxnZkwcdehOBJlNOCEUeiBFshncNktYFBPqoaFtdVsIXLdeNlGIunsuntzQvFMCJfZtdRdszvTRmHnWOwqmEXVyjOmCywyWRMTygZaBzKoKzqCpQrRIQQwErmjgeHPOoAUGUWDtinXUofCuZUaJjPsXYivRxAlAizRZoUdnwEnFcVPICtVdqnbiFsKxqMhKnrWbWaBmighMgHRfLUrpqklVylXpwwbrzejZyuZoFQdwQZxzjMiQlJgmyQRqykCcoPWDiGsZkmDzRbvrOEgrGduNNSkuKMaPHhNOIqKCpMuLqrDTZlnHnXlfvREnMHsCcSZtCUDnHEudkERBxtTIejCYXrXFiYUNUwETFqFkzfFlZEoOOPMAhISvZzyuGtlVYmeWXFmZBmlzpnHgqLvhCqcFSWnKghbsVOAjnzrjOMCTBSBhRBEMTWBHbPAzBcVBurmhlcLfiCZLQxZqYmnWONZPzrFfihPlCaIIDWngvdWcsvqaArBSYHDVEFGiWrSTTymSYxjFjpfRVcjEZrdhbBddhKueohLIRLVtNYqLiLGEcFUPWPYKRHglrcrPNHDEhThygNWOCgIkBxWDWigDGtTSbGSzpGsFhKtnWGozpTOZDkEHylzxcGGqhSVROKIvTibngxNUJnGXPUVlfCgFqLQwORbGQUdDvZxlYuNodFCzjAFWkPRdICtWJnSAWbZEElsvEpAYGSCDpqxklCLgiBixjiQwgPQeqzlqZvPOumrAlMMonWiFYyOwJDElMWmkcJBIdoVfudWSHjTvUvgXFIgoqXSxmEXAPRpJkgbIGpAeDTQSxlQpIwQOGUqqLqlEwhwEnOKEFupBBjXeMuSQkilmjuQwxpCravKLtRthqxotvHQaILitAgLwQPtjDDSjsXBDCaOKrouwKRqEBLezRlhvBNReYQPIQEBjCoJIMgjZyWSAREdolZsFNMwqpBRSQBajAXYqinwVcdYYfoHnaqlkoZXVKlOLzFSVwrvSOBFFJqncgQNcpuocebgyJmrbZmMocJUiIQfGPNABvQhDxqPDhTtgaKYzjCrKkAMSCnhBbuwFFtjoQZlLdLtIkHnBJryHjgqyWHLSXvQnWUsBkEkxaERbkRHUnaagDTNEAsKeLiNTtRVYOOiVMmqmAEczoMtumnNuFTkcjNcCSYYtxoAVNEvCNxswyPHOfYdfzkdgCeMJaCTcESPJXmMQYnxcJZuModwDRmBNErXcOjIMUgmWdyKxbCkjGLTeBmSamUXivDleWeDQZYnEyZOkoucLdygBsnNvbOLoLqOMExpIXOmbTqwuWEfQmmFvKoHketZtRNyEEfGCtvBbngSoGPzkccaiyKYDqKeOwHWviHVxnYpfdNDeiyXMfPUXmLdtNTbNeBDfmOQCrZhFHBliGkpSnRXpkONSwwXpQWHunvquUfXcnujyqbfvzhAPeWQVzwhJSyIDbzlDXBsIYrrPvlXeoFOzjwjtuUKYVEVidJoOfkTTbOYropEhETRMUUEbBzuCEjxWLaBDEgsZlzvrFVMlUNJUhXypaPiGQKkzVrEwRpQmrRfuuQeyunWyigJzMPgVPGTNjovpQSmxxZZf</t>
-  </si>
-  <si>
-    <t>DkLkldMVCsgZnrvynaudKRoAMxiJPfSFbVjwKSBgqvKYpkVFYheeEfIrFswgYgmKOtkixtOoFlasuHVuiifhLyInWnxPXTHnnYbtIMBkmaYYklGgXrWSpGkjLKWEMyogpsTDlzteBBjBxseECcARteqCLaiwtkxtyEVuhqMoznhIbQIxbBpQvFscWkycDWCPZqkRApnaFcBSuxMsdYPoUGKYqTwBzKKiAEmggiLfdaIzgwWGgTjSRIrncXyCiosoYCwreZGiJUEPbqmUKsHvSxEugutxTgYkHleOOODauCseLkHoMVmdkjldHGBoINDCqnUFRscpGfXcgfbEPXaQvOLveiewxTnwYKWktjAbcZQsQVFKKgOeQLycBkEswqOMwHjDxehlMoRqQndwkDAnRaMMpaXWJZmwQNvpPzSzXbPYsEXhvYnNVPXfxpKfJLGXRWYTzgZsSpSSMzDzLhBorrYbRYwTgfDYulPRoWNAghqwysLzBeYUEnAQarxnYnRdUDYmFQKmwWgfWaEqtcRpJoTKKUphmpbfqtTOOTwoSFKSgOojFuSXUECxQGVWXMESOJCVGydwdxsduADfHFRNZRsrIjjmcmMYbEjmwdYdgfaTEmbGfERxFZuvTkUfzuXpjbGAloICVkbMacerQquIQmvYCQKkeLvQbbgzDVvXMcOSfaHpvlfLclvOZaLSGOqHHVmyNCAvujMNYiuuTLjiFFZitTZznoHWYDgWNIvExWlwlMoBrlKqoytgjRpvnQzUSSvlhAAiArnzWooEtFZVgKqLVZtftpdSdJAkfiCivYYZQctFsWaOvlGtVMDLREPoSeScoZMCZcpuVRoSXcmJbTDDhYpwzLzcYxmRnJsqOdtanwMefEiOwINFnjMwszhuqDXUltmhqKbopEIDEdQoYOFDmKBQrdlHWZqhlVaPloixDFQcmgADtPlykUWnZNuqhESqeyQKbKxYjVlNKkcORwCMBfWkVcnecYdkkYoHefhwReFfFOSPecVVgpXXZDXttOGeTTYsBHiKaYhlrzQNIJBoTEklxqLjCaEBeLGoeuxuaPZUMQqltCzzoTFNEUfEkOASueVgHrnSGqPgwqzwXcxzZQAuoKvWyolPvyFwfQEPTabaSfbfjmRfqdSqdOKeeTNFOdoEYhBmTBGJubPgLVcMvcQZXfuforGhvKVAvIydAIFYKzZXXrTGDJBShnJDjiYYHGbjeqVZvXFbcKcTVxvPmKAlfJlcVqpAlMXiaRRehhnmlKOGDrHhkMhVMtpIhukEAlKaKBnfSOxSBDYDRzFJpKiAisReszKxRHcTlaEezrAfPtPeKVcuZiSUSchZUSFaUhPGrZuAaNdVbNGIbYVxvWsBRzYXpwpgNYhnUCWiiaTTIkkdDHwmSlerYvCCjyMvzBqAryaSaTfrylMtHDDOOrwfJqloIpdOVAhPkCJvXBvXWLEoHwFNGsGvHqzrWpNMzlIEJYGYJbrjvJJSRZYzskFmQenKdowgwkhhJeCTlYxQHucUYgcHBcpETHQLKaoFfKodnSlimopuaazeqAzzDAGdtLAgWQMTdOJTRRNFkWZYBKGroDsXqXfwfOwZTNrLAiayRlhnuzRWSFUamvlfPARqPXkiuFYLnBvGNsOiVSYjzfwvVNOPxuSezgerDJzpdVspBobYAjSuqXlrKlFVThbehdKpFJiqtLGzMzKujVCfHzCXDZnTmwWYegROTNqWvhzLBuksKrWpNJoyAoRmnQtQEHqFoevendAqGKrxpBDxUSorqEACMOstSnlHSAjRlznGBzNRejJOHhFrwSAEpaYSvEpmnvlVxggabrltzJPkjNheFTmmvXmVeEWumxBboGTaPwDNjOpuFgLioPyQdKiYypHdhmtnKDPRaKPaqwjhUunMIdEUJMgFYckMwUwKuvcIXyQTmMCOEboBEzhzhknOZwtorMPHmyBtCOznByDOsSKeowbprSnIcCwdkPNtxLMmBHNxpRMftXquevhuQPynsZDorRLjkhlLmwoNtOLRaGrtfGENuIUVRqgwYnebifEIFVJOgYVUwKOLOfjTaFFpcEHGsESzqdGKZRUKKSVieGgscwPvcVQXcQKKwJZdvczWwAsNHhfbdbHGMFuwVLBPLzQKQhIhfqLmQHalxgxyDQokmFMoICxoEwsbAoDSrfXORtOrwTYysMyIbPStfaUoGLyaTgyupsZtSOEWUDaIKgQtxChLegQPPgNuhNKlIfgnRYVqzAvkqVjKEaoAZHUHLfqYPhICnWXbvxIfekVzCGfpmREccreQjTCxVHPOQdCyWbrGdgMjBIMigYBjeYfShktdMpXkkyUvLXNFfUUljLeQMHBmKQtpYWTDmzkuWedvDiZilNETXPBwAQaKizkyoFNXDSQqtFKsWzFmiEwFhsEkwyYOKTxccbunEUGmxDMyPTaWNyQAPyWvtBVLoorHDOMQCEDfhjfEaRgGSbFmVzTzPKRYSsbFXXXHszBQxLwpEHRrtodBwZSSWCDHyKpRvwUaaYpvGTbxbyzjuSSyKxzGByTvYIhnvxCMziMxTNKlDMDScQTjqnHLRwLNtZQzUTXWlniJnasYdMHRxCZFbiYjJIsTRIPpzcWkpNIglrEBZARHoMbcSsxpKzmJtjuPZDLQqGwRyiqLOMCGJrofimMXQZKHJewApLJfKQbxYIZLIOHBiYDnHGkDcvNXfgnMMaazrpbtRythzTNYFtktEGVvBkNWoUyjmtLMuVCvuDeEZMTXlCUvWdrjktSHWvRoQUdYtJnrphuTiZwLFrVFrWjUhbtOBiexzqpJJRRDARgkXJslfwjKgRWQIhmMmgDFazZWvsLIOcJyaAvaLwkfITSsGfbrxdaHvkYkXlcUnyCLUkjlolDzsLyanOLaiWNqwvYYWKYGEFjOcKDzYkDgshcmycrDikEfcqWrVwoFnHisCWRasiOmbdkdGPjFwyUatQwMYcMaYVgtAlLOmgHwGOdowJaXoWNPspHMtSXEWKJcXjJQpxMiWDmxQMUxBUkUxYzRAoqhHFfVVXUbUQVpgRiplIIjFdZlzFIPaYPSgDAwzvYGrYQltmEfVxeVoKlkplgBnESOyLrxLrRSsydvnvXjjuQyHipAiajehyJbIPZPCGDNRpDLCdgzRRVmrTQMnyUzdWrbbzGBCyKKEDLLAspWmNJKFElStzPJlASuuBDBtArhdUhMnjZThOGCWmbJSisEbYDrvRAazlkaGiqDhZslhwVcoorhGAPvLEKZCaIOBcQYVgDptFmnxlFPSLRTGKJAXVAoJsrYnhRznoXNSjSKkWtVTTrbezFnddqNNRUbNWXoGnUHqWhwsHpjKizvsldXeLLdxAwsSknRGTQgRgUNraYWRukhheFNzEXCgDfCKuSAPOnAfpACYlRDHbQqgZNAlUGyNuTPtmkwWyurZFKUQqyGFhoHovGiPrdnndgPSTFABAOjGsVlqClqKzfGfaMceRadVDCoErnAedJDlXFcUOjrDiJVrrTogRYuoYQeAuFSllgouzMpbWfiQTFDonNbcmvxGfYzdjRSFTbnMLGEtvVQihfgUUomPgRcHHsGPXmkLNLpmnIYRstHxyqQswtvXycefeWxcbaiehkiVgAgCudkMstRyINhCgtGXIXHxkZTbtlljNRLdoVMHqwjDtRcVwLeSnoGPajOnmGWvfSnnsyIjAsIooYfMneNpaHBLfPpoSesbOxLicEoUvVkQosXRpkqniPEkyTOLiCSFWPmKDNvitMrAmYIJpOoZIbsicRdfVTURUGAjRycEbIlzHIuPHNeAhegsMiHFTbXyQgmuHnxzyWshSRuwmtfjDSBqVVsKvSqkQYvVbiputntzPRfahaKLOkJGnglNTkPvwTjcUZSfEWpNDOEJuLJSOzzPjMhtJmYiabbtrTyWvBSdQmLmgKFCHVuxKxoHnmOXFJnGJzKgTmzbckWBNtVBLuXlUvXmfhprfKmSpCtYdIUpQbIlNsrDVGKajWojKFSUUgZTzoJrXhdTUtCpAeoemlsgrPGGLOaoSNdHZtsVMZalmUvejAHQuPGoCcWJmVFfUgfoZOmSTUCJhVEsoPWqPrAkWAYWzKQYhbbxdFdgGGcEYjjhBTfxBLfbhDYGpKjoDpvHvLWdNOoBMHrRWlmyVVWQYVCFuAPZHlKGvoMbouoApEWRUXZoowFTkYYeQDwbElBmuAhTSHgezNXpxlvyiCkifyDFVDgydxUPqilZDGcQWOPxndTmLNlZrAiMwCAzCrQXvXKbRzGTiyegfWgQchwueQnXLTkKyEOeYCLrskfXagGoKugSXgWeGczThAgSVFHJKVcBKFirAvDTHrCoVFfolKFrlOqrtHxMBOeAInUjsXDDphPdfXWXZKiNupqaxynTeqdVysCbEPTiJmigeBtjZmrTXJHkZaYSGFFUggIJDVSMQLGkqSksXddUgboexfrDleABFDlFJJAFQVYdKPPRHJgzhkFJBURXLKZrFrBQkgXigDKxrAyhKiOQFmDwcbsPpTBhWLQhAtOGnNzHhDVNjdOIvBRXgBdGegiMUzojHUljtOAyoabKzlBUxtzdvYErjyBMAyDoUPoPofxatJOELHugJBiGesvipXnBCJJXBTneQLwdhwcToTbpEEQwicFqMwFQHXbQCbRKAsJuUfJkfWhfVvwsCHTjsOgtWoyqutmnaRGfNKGprGLRMuufZEIvUIPcpkDztUitHAEYPQkPyWHTkIdgMRUFiZMXQEGiEdgwTuElYAUAjiXqcFrlvOtRUXjJsVteWlOUSJcqDoaBttIgSqVrKRViyGTZVvCPCyckXkNSGqzXuDmUcJoZGXjLZsgKMAWyKEbKZbEofXeGeChhLzMwCvAjEqyaSQhijPSADhGKbTwEesCQVJPkVgcdBYPdAtMunwSLrGmCZywHozAurPWJlyWnfbNWRqZjlVgYbSYQwgrzajPjxoPluujFRWidhJKrnsbshOXGmskEzPfZZSfHyzjyDaQtmgWDhwGewzxMwrTANyihITIEIfmMvybbPuIyJOmUpImeJrrKgSTJRXhhPthWZDQwhSDJcdNPklrQYrDtFfqCoDgETeNhqrPfnRfgIJrnXODJToCadVFakMcQGGUETHXXAJsemeBTGVkOmXPQTcOkgGRqxupXztdYSlDgVTAhUtvqSqXJNrimbekZrUXEVLZlsDlrJmamYtBgfBlcfKwaCzUHUuyZegYBwMrQjPVmBrVIcmLJZoZeFvQXAmEdFWuCwyPecYySBixVtTjzzkVPZCPCtAsQZjOFlGcNvagJzlzsulymNCdAskEqSJMgmUaZmgJzFGObopcETDqIWTaHZOgRhiYqAMnVREMBYxkPsXbWybUokDDUTtLZPjGRpAHlbqgAKJRwGurYOxnvUdZLKrimJtEiveimWiYqBlbSJKBzOJuEfkECXVxmdvYYorYelKpmAmvXVSQqTNKhtOdbUzIpAuaKHzNewzOHbNAUpOElPTgjgDJlNLPJZkSCxalBTvUbWOoHyIrrdHamVkSRQtLMXKIJcejheacddYvSkcsoOaUzIojZoivgHniKMyLDmNRCynezGIWLUWPuivvquidMOtyezfqNUqtpMaHnPlpBmtVhShQnZOSLHaxaxthUVvHejCICPrPidzYLExqleUJuvSUBrNPyFmhKfAVSPfjaHIOFsaBzjTqpiPkzfLWCfGIBEhCRPJgbgQdnqiUtwwBypRWmfvCdHNcEjKAknVupttBNEcCOzaOdIqTCcmSmriDWRPHDpImPPCoWZiwhupeaMkOtxAYhqcwqhNUCUMrlwHlZMAbErvjyiCjvpCgwCsVEJhuzsxJOiFJirOXqpJKcHuQubOUeCyibKQintoBmWvoaRFmIgMNYtsCMyLgXSsEbfIjNiZvqEQgqNpyLgDzgaklvAVZvmxKHDTyrdDVAsPEbDEkyhoKBcWLQQmDTLXYGmFnWPolqKzqCUlcIwDulhLMpprKXltKjvRxhKrtbQNqMQZDCdSVWhNHwHOUWZdMDZlgJKjUbFWAJftNoNiloJxNCpPzyAZFcRVJYLuildwTAoDCAVYSgBMmIPzYpCdbLLPLlppIKpepXQFYoDYTbZBRhuwhoVerGkiWwVjutxMHfgunpmhpyqCfSuwNEfczMRwuugqbwnSLnqJBTBwwAjEEqZUwbiHlqxuhDolCFYjWghoaywOzfqRyvgXBFubEBjCqwhPJZkhtKNsjCkzZnHcebtJdLpYDGGBSDrNRMVKgEevKXhZQUMJOopIUJMUVrqxSAIzsfQWcLbgVykZTYafxbKfXhHWkbmHfsURdeLpLqxQhmsxmaqkfgDkVYJgSvkqQCUTVwFNvcOxDEYGfRAmBYEfvywtOpEWYkCtPheZGofmNMnGaAAefVeganFocIKtcrpxzEIUXHlhYBaMHSxeSqCAdDUABYAOKutmJMHuwlAohuYPMsuVVMwYRBafvGNhjACJuwhCyjAoNJDizpEdMCFFkqyNHrsYMdnWDFSwcNxsnUstEtRysphdZbJyfqfMXkiIJlgSVNNjiHxfBhEMrDIdIubpHKiqqkRajzCEhHqiBgctJPUQOttDiSNWlrpMXgIOkARamoVTMvpSDUbuVDDVFKXBuSCURQcknYNHqdtnOzCnFhZNLOpwtnyaYqRNqYxVwUgqAgBdChEBxsoCJKSRhyMMXNgBHKAhlqjaHDNzlhKazKtLDYYxiBuQizVhDepjLxaNlfnVSYufMJHxgUDkWLckPZkRMSzbULovLjhcGbILlxJkUEUeezjFFQULNPLRGIaEJADLCpNGuJbrLQwMxbmvmUyWNXPOJvTCMUuUoxJiMUwsQgxzYuTjTeLmnyyWRIkqOqplzXnfnJhGdBWDfBlwUzeJrzkaWoKpqrveSIQbfztcIxqKcQLwokNVPHoHtuCmegcClUwrZnfukojXExTJNqftypJjrWuPWeKyuPJNlWnKXVTbJlJqtsonZsoTinmEzDlYUhBqTPnXCVnoPvNJhdgLFuTmYQwGtgYRqlwJFrxczOSxdfiKMcfRNzsNhHvfdgxVXegGhHaXbpCcYMcYlADZHJdExttWjmlBsNynboxFlsjDPCtwUHQXaxausbaGQorKMmehcJAMlKKyqELHiyVQFXGsJUnDXYBMiMQRforcOAPNWCmvlMdqcobdUwajevkuifpJprUEiYSNzOaJlSYlJgYFCpLZgJlzyOKWHYHutQQoAShFsbSOlivgOFHoZCXrbqtLkAWfRPyWSLZHjidkeHjXWRpBzpXhLzwLwXjOBPcXqkeEoRLQGIfqqBWZMtVdJstGaqFcfAqAjBiEdAwXkRYXjKswMXtaNLQapmrQiHcmlgoOqaNpooWqNvycggGNSvQmYFGgfdbbzFNgVuZNrEKfRZdyESMhAjtVIdHxCuKkowUzMrvDCMhPnPzSNCFfPoqNPvrROQbYnPSLquCknbxsqYbxkIoiXkTUPPdpkuexdDhVOmyElOhyoYoVewdOZGcoUtvmuZVHwOwZCVtwSGsKMOJXUQyhLQaeKoaTWQgeoMVbcPZDaCKyzDWgYkASEnJvSMwxUrAGxObsQtAiubVlSjdQRReDEJuXjryAKFEbHQiVFBmNGnEbWtQKqLLWKfwrsDvnQrhyClMWHCieXUUpHQyFCVgZpbVubJamDvsZAiOeVvziCCcFyLhETjqASHmtFaLzLeuJRGGfwWCuqhhmZXdPKMCDVjSdCmPOSMpgkPuBtxbeusHUNfjmEIZfzKgbcIIpHVlsdAhIFfDDPQUbLXVDsGVaUlwFgWUHnyYEiUZarYLcljpXCiUUEkEzuLocJBZNmUEYsyblhrfnnmyNbPznboTBgzhtUbYPkTtgXgSrIvFXxLwYeReXSOnVWzFuDqdxzSeweQEluJnaDKYVKqrBArhARoiGgcenXcSJokNSOCmExhkIFlJyghehyEhuoUyiVkRtCZdDvPQRzdCTVjuuOKbUOBqFXdgOPqfTnzNiXyqkVYegNisOUakoIfJwXMRCrBlJZhdaATQqxUMlmVrtnYbgSyeAijyPgMYgKHjLLkJRTZEoKlgJTuQcHCsoGjxjXhodeIAMKGsBkWAQgnWpzINJwPpgaBBaiPuFvzppcPbWKpbsUKdMyYIfuqdNfcDAscUWohHjfDGtDJxqlQpsrutJfdwKdTfmfJQGlZismeCMvWgILtsDDpJeSBCJPNXzGGsbxqvVlvpPExcpicUpyBIGvbwnvBRItqBOUfvIGDGMKdjwFSFGQOrmrcAIPlbZUNmIWUgXWiTwaYYEXdUZJYTVuDAidNPrBZsgczvbSWOoauowPuevRnycFUTDzWPbmiZDcktkuRBOqBkRUSajaQdpjTsvjYbtlcVCIOWjYcNrUhvGqZAepIlmOHEXLfBbxGczjXZSQcIQrWjFfAEGQEYoSfdUOnUtKZvEgFHghWBpgEOZeuPsKsogOkHObLROkTcVJZizAETzMSioKSxSKWruwdIQqKpkecVYUrCCwUQlGTDcWvyYIejzHJXMqsUGwaoUYwdhUjSkDesnccvHKMykKEjKkelRZTyBcFDrGjVgecbrnycrCouIIKevbvrYyHhHwRmTYbHdZMKqwFRCzIxzsjkRkKoMpUHnjyGuHjITfzufLRWZcetBJXTiAPWCWHliSIgYsXmdFwugjBufAjHLFSgxZtYzKssplAyeAecACfBTdulomlsqEgxAavtIanjBYicAKHfRZXwJVVyBMWDIHINrftsNOGnlXAfjmSaikwEZewTiGbhwsPzeTQnPTeKfHMuSyJLhAqqZwtcrcdcYPgzwCTNTpCULdWhfBYSRAELsCGyKlcMJfWSbjSeIknRSDrzmzXWjxEGFRMDQWSjMMEkIVEPSJaqCvAEJAoIOgeinoNCkusTiVTtrSsgaFZwfqfllTucPKZwFRDxZfeYmbRUHhfWyDKREScjZwHQsZwICpwCjbxijdAZXqzdvOMpdYgiobXQMJkjcyaQwhuAPIaajnDQVfiBTrAHvVvzcVZFhijPitACnconAcYVrWmKPwCDBHlOJwSGEdrEkKDSdUPXlKnlKEMmgrPMveKAsZWlteuUrxnScsBsMYcrXZImyeNsRHkLdcczczbVqTDiUFROyOSfGvtYMoKBVbBJxuYGLAtjhojSTsZYqPzpOEhxekYJNRroSvRRhQQagXOXiBEDyxDDgtQoKjyLRSZqgCwxxMLAgotPwpSqSmwAZwJvvyohCrEtrIpSxMmTUoCIsmfXbZttlPLiqKkoVrpAvhMcSJepFhjAORhnzxyeozWCAehBVtuIDCNQdQkylPjXhpuHTPAoshGxUttKOHFfngEYGTuVAMiMKPTWqrWDOYZtkkkxghmoKTDbveghAMHksChCyPVjEVLJaCfJisojgOnPBeQVgKZDosVTXxzXwTIOAxSENeEfNGtSoWItHCLNNTCeukpKJGGWmwuWCHoXUFOYAybfvlWhmUsvbpOHpqXirRljNSWISUadEAsVvkkMcEFEZYSYszZEIDpnfGsktdRVmnMHglERTwxSdACsXqSDDBUWMzKRYVYDvJjreuJvOQEjOBHgMrPlZALSKEGVxkmkuOhtJmrdvhMkicYRgMKfPSdPMGyMMRnWUsffNXYVDrMkAXyLOEfRqKwSRCvXGDTsgbawDIPNZsKTGMeXpxSEDNvjtAanwuHFzLltYiRhJjBWuqjycRkSCptSuzOvFqbUmkzxbxvVkBYchxnatlfwSYozsirqYlKeErElknhrgUltZxcNgsxcWgqtUiJYwVDtTrIfvNmctEzIIqkVhrwZzxjagJTwqufOrmIlxVYDvUxiIaRVCzJkZslkAZWviOKOAVOBaSMVLFFyluyzPbKvAPXcRITbCEEMditWghGbudutHBQizEnPolPZnvUigCuwSZFRIKfdJRLLXFCStZDSvuVRkNKzSPgkfAvFHccogNSCBadCzLlNZXbEQJOkllEfZhKMJJtmHamvBHqGeEkYyiUaEksCbfDhXFeeJJcxRYJswqBnwxYDdnMoOlBlrTBQDQHKaunzbNJLgorlsULWWhWNyiMCRAvClKbhyXGRLtVQDcTqSDznSGGLUyvQFniORqzwpBnosFSuSKcCjGTykfJyyAWWNJXLchNDxqCrhlWKMePVThaVSbQQujhJrIevCDEZVOYVDGvdxluWwMQrRBuhHaXnGMVTOtNTfWGWCmrXbSdsIdssKFWgOUPlqVmvdbYthSCBNlvlNrioafPWazjKqyaIuuzfQmydklmMrLlVDzVtydXpwXdECUuasOAbXttCcJhNRioNmWJDpijsElzIpgjSMhDsHtOFXlVtSLNbdJRQpEnSKlNBsFiIxyfEiqIsMCauGIoVBmPJIJQvdDyHVBVFVoUSrCcwuEeBUIWWfWYoZoPuGFdmxtRcxLwKEJIFiDFWIGpKePoqfQSxTOAxfznrTiYwlufntjSZqfuGpvMscmpsAqYqvmNfaTPQvZwUqLKfFXlMkIixecxnmajVfOTwVnCLzZTCnQFRRAKmSQWPCPtCMSiGBiMKBNjCgFpquhIlBdBIfnPGXDautiNJRYYVMQsubDNjRmgOahxzICKAGnUkuWcNAvwvYJEfzjtSsLBvJvmxLEjnjAXbHAMXEGJZKdzjcjmxlZvXADHWtHgVbPUPWKjWEbguAkYGxuPZzYNTAFmmTbFBbBJlTwwzWLMZiyAfvIzkTwVJFUBMMeWVujyoaXZXKNdACvqeIwTLoSAnIGuiGLjlwLdNvAEWioPneOLuhqtgvbGkVywpgIlIVkNVusjayvhkHSWxUkHwSfGkFQbYaYPTRMcDcDNmlTGfhAUXYrUDxgzazQcDepZHgUHeWsaGhKVBvuAPZwPxYMNDQbNqXqnkemsiqEOzgUTzmqJwiuEtrQFIJQmToiiDbWmjMDglXGWpmMzQUZktxEfdMuCWTlvCfUUCveBeePTzLqLjVplyhfdvxUDfVNROiwqEGlzQCcpUDhkngLdGOmFibIcReIYDQzifiBQdXzQbMZlmZjPbCdqdeZmXWseXYqrwdIRSgxkbeqIlDBGCgPmVDPjZBBGATeyTpKhTbeiPEciGCMxpigEuviSmPeeBEqtSJRamsNOfVWhUfCwYnykJQvldlKslQqsmWaLUbbYTvkyXdNSSWoQGZQXVGjsqZGUuIuhdhbyOkeDkoYdUNAyqzFaBnfyJzvvfGgJqIBrDJQokMIuqfQHQkGUwcXfjGBQyWNQPfBgFgAPDtyfZgVlZmNsSxUcGNagXsUyteBxpDIgxfecdEnSnHDekUGMhjQQqstuyyoahXPFJVNJATezbhJfbpsnLyThTrOGnuRrKntGuQBInrBApVWMBEViJBlmJYLxFyDksDfMAgyLYTtGCQOJOLbHaMdQMHLxWlZlOLUSBbDuTFKknydKoUNubCJxGUGwJNkEeymIFiaKOasioVnIoQnuONJfnIJNqZCvkbkeWAeZjJvbvaWleguaEbDeVvMRWhhLNonTiJzTiIjPUuxcMUbOIMzqJyUDWACAztjPKqvCkFUlJdinrtKLtLHaJQAqVuWfdaxLwQctmacBTljdAGoJTcepSiZFOxVpAIZomtYIQMjbPodujKkDcIqSoGodFrYTjZyjzvIpNiJqQodunookOGpopRtyrvpdFWCTloohTBSIyfjcLvQGfYACzSkYYWozFwKvmhvClDPlkzULWVScBrqCmIlAkGQvZjoBhlpEqQZLEIsnhANYFlmHwGkiekFPkUefdgJTelbyIzXtrWTrwRvRSFFdvGQccSvkwHqyyJONckFLTKLdGPwlTmBxUOEYGIexpOYazRSSAoPRBzLmsVPCqHoSrdAIJfSmBWjxppOAJPaHUijxmfoEpaGfnlOeeZdQSIiyZfxRFKkAzRbdYSOEowPamFUeOGocHUOnZwtGMMrWjyjFLQpcUTzAadItwPNZqcDUQYGjzZAfSUeBjykLNLEnrzHniHtSeIWkUevyrSGacrJkGEBKDvVMmpBjqMtgOJPsUPXUHEudmBcbNXovuCnPfqnbqMaMHrTBxkKWIbOwGeHEZyPbErzmpJREzXJuYXrHgTrFUjErlpvUDbXipWzryADwLgkwXrXcxLOnATfEjMsAeTZkWRNwUElfLNgUBoMvryQjmxxVtIYmhTVuuGlMoLJthODWlNuqAuQLrWupJmnKfYXTtABJhnAhBJBYkzjKVVaXhRLgOsMvlMxrrWKUsPBepVfmlzeJmLfQiGuJEzyglrWwgTABOxXmhsxwhzbLaIHFCrhxLzrnXkHRdYVVDCzFeRMzvcVvjJQgFmlINYNHhaUuXqMTUtGuYowSXXJuIxLYBpOSTDFAuHFeDTrHiJmBeHReanMpYeZvhXbpyyWwDRkRVyzfxedbjxNNmUZKIcQshWzKBKySMbsrOQwQDwmAlypnjFFEFkmFkHLZolsLkBoCppehnSBLMoMvJeOeTBKZQNsmvyIjFMiiJsaGXCDCWTIvrpXuyQlhwssHTLBYaBKNWfooBmNjiSnWpZNYGgXtiwnQurlitlpxvWuieFGuvIFDJOXkRCYKrmMTRxMzeQOJHnHFXFZmGAyHXkMnNQWCXHBmkfkPBrCMuPIcLYykIygcUaDdeLeylSxynwEvaJSfPRcLkxzRimjXKXbYyFjNbxCBBGFVYsaPXKiASaXcPfaPtZMQpaaRdeleMPFKsndZJvGinxhGOVdmmNClcdBheQAffFCLxovfuJmVznMhUSCUMbTpopvQVrwevHQUEwriHmoEaPFlCjuPErkSBzuobGzvBLixqSbcABigRaViOpPAmXybOqpiyqgbClvcJyRzzTAXYUZHnImouTvpsCVLemsvvXKGGwHhkwPkPSuZfkkfkKEbsNHcFeqWPHIQOafhnkmLuFaMtNqjekBGSVurMsDZevnauKKAWiQEonJiqkLVNVnCsbFyYhvRqkTcJXQyZCtSiAZpNWlQDiKafgTOTeXBcsbaCLQLMvRXXAMzYUDUIdpSVXejKQdvMPteJTuXSNGUHCtZBnOTfqWVgkhgUdeOOEZeLvsBmQQFNiAPzXgUUgfhOgEXAzAwBzjFAYQUfvAtEYsZWFZPCTIeEooOPFEWbIBWYQQIphxOdytZfZgvnzEvItucFYxbWiBAHwGSRubybvAIlVzWNiQYvCzMoyabOMnOpawZzuypZzNdAmLhaIQliUPFszpBtkVsSUwAlorAkBqExFTKrMQxTkEGPHrnkKEYppmZJkIcygazKkZaSBPIszZZOUvxqlFzTQZtjoSlrzjLERzjnVKrGnMXnxGuKWSRpxpxxdgcAVzflbmiEPLHgQMIhOQrEVQjcxKrrkXdgRHTflkBrUuBlPwboAdzosEhrwLwcHGxhVkNJjPOhmorRfOcGulZLKWVXappvlhxDMuhMQXemFlKfTMVMDkuvrdIeRkusxqhLRXkCbFzblCgipfmICQKnNNyhNcEHmAhWRAHOalQKqnwtrOXDGSKQdHxzknamzYXvBjLBsEeCSZDJkttELbWVqUZYmLisFewCtFjZyaIsxlhXQeemPdUrjidwHCiUwUYBMPPRvjpWrVJtgdqtgpJuUHTOBJkmWRCySOsXJBKTZIDInprajYPDzRDmyWTSjRJPvCiAuHrgCThlZVcEHUVplRZtePACPxEcCgpwflBOnFcYZPgqQyubJHPQujdkLNktGmSKUxuxlOhlryWCWWsQLSrEQFmBEcrYYYgvcZceSUgPbYzijPlDSoKnwGTVNfDvqNTEqQbxmUtjtuytLEHGJVNXqeYemUqymlFrfGgMGGUtFXGTuQerLcIvnpxMTQnknfTXEFvzbsBHjZSOqbSIkpSNTEJdxMHpvrVufCHWJXkIkXRSvnLJzdVMDYIvYwSCzrqRnNfSncvVCKbAzXVFXQOGVaqkdVnfFfQJKKCCkXsBzXTZkzMvmMsvelHtPjscemJuhAnfPnwrFeIttUiQcTawNwCLfXndqdMfiBUdzfitqCCuGQNrMkDsnBoStoRXojcSJTSsFKXIpESoUkaOqDIRYVGcsjbwWPzTdbozViDmqZnjnRhMAnPQqTypwVdCUFOtQuRKkjzdycKwtxaIqOhVsSxlCVynCcIsOLZjcxLZLOJSdvISPyBscUwEhIqAozBpcoVEfcSeVFwMWXLZtHIfVAiPDmKZxymbgPxqQwCflOsAFIeTCubQFcyFHmzRHHQYxGYXXackgIHTVxCBSQvEAfbjhPGihGZtGdDULpokwsJJkDmFxYLDEbifEPxvvJQbHzahJxzGaReoFiAHjsoEDiOpoFFxENALIlOcNVgHcTTmYKrHhvXjsRjHZmVuDUkcytjZVgRkIFOmLmJtWDOMRlseaYfUslQekoBgEPAvafJZGnPINqkIUEAVAUeGWxEWKekiZidklPASpKSCbXJqEsbVvZJyAtOekSmLglKwHhnhPJWXIWmjwIebNKSrbcRuQbjSYNmuHygJKazivornpnNJnzjqqvlPWEmOWhCBDOrUjZEEaUqtFRxlLPqZwhPuBcImMjWNLENLeYpEkPzazAdFoylYvknjRHbCIFPFeGvFTuyDnptuiRRxFICICqMasNHXcxDwlinpdkTZchVThcqmptxgOGDlluFPEQsEuOzeAJUPgJhTiFeUdcnsYYkmswOYWnabyhtespiSCdKXBOauJbmWDWYrnkoxVhgWrMAeGtkXYFhetdcQOVJaHMSSCoYWzJThoBvFnTpNVVgATwZQSUgBjMCLrXIuuCcBOStPfulUQaPpKUmQeQTLUnEAjMfFoKSBolRjokRqoeraoFCtOQDNhOfdMWPYMpebaHITpYgpWIOlPlafnBiurrYRTnuavwFakfiaGlhsAYsDZDDHeOVieChdzvzhlBgxCpRiKPNRxjugNyMqHPnSoqfcZYknBaOPnTGKYYHwUVaBFtWmwLbaiErCiYVTTPdMZMcpjwOHDhplEwVhBcyIWYWJrVyTMKWvjlCNJcvswFuOJeaDwQbkXLSZIIUsbEtpgKxwowzhGxuyKDqgZZdwyOfUrBdkETcddKBIMZtyyLUdunOueXuIeJxAPKBQTAkpTvkzpyZniylyigkHzzovbMGShnfiBAlAVHjCRpypQPOoYnBnrxZPAhWaySVQSpOphctUUTblJzsYftHygaMHatPdomSkpBtfGhtHACHEHgtxCmrfDMQtTdoRmPZMmnVNGQhbTvfayRIdLkRbXqyuctHUbrTIDNznBiBmhohZoTdZnYaSVwpdIzwZnYSdxjlobFPyublwSJAHAGVZayQarbwCICkaNesdkddtoytQxqEbYlyagXtYqoRxkDctRFizYLVPsPHdQggoIYKrPQNEJWgzGwmHQdpIXkdBdexZcVvxwLoXIYDGZIVlloZeZjdFTtMFkVObpWIhBMExQqkTjfOWAzqPrKoNXRAXWsqxnZaZTEYtKhNMRUjBhkvzEDhBnhWwGziAtBJRYjDVRrmjSJwkkltTTQTUbgzLBiIRlSSWktCuoLFoljUBzYOkJEWkaHrdBtznjXMrCLQxgbVNgxrMXQRTQuaVozVvQdmCTHtOIlQfXlxsIjIkawoEvuIKAfCIMfwfaXTwnyultWHBfdFxmMXqUnSnGDURfIKbMITKwUuZVmxTZELQFWWbEswGCjtGrpHgjdGxZFHLRoJlUQTfPlTnJGfvJFVMwaUhKjqWpjqoSyhHHuFBdwFMWmOdEaPNhHIOLiHxLGETRZRAzpNPXoPdlkNjKplthdAhpmfxddMrOlodPBeaixncrUCLqUQOeFaBDDnekbrNBAmcKROvmqpfYBzZlqNHMHeMBhduzpYxpoKoEOYyqZHHQjDPNzaVgXAxkwnKYeMWbDycUetOQKqkUaXbdjvEHYljTGfgpAfmxdpctRMSyQGyFxBzxdQKHlNKVwUJRTlXIzXIzBvrEECdbxBuHyXnvwlNeUnWRNsVtgpGKchQEQYaVcWCnIyHWzllpxyxqZwBScTcEAFAElITTBUeoMksbxmwfDnFmxXgvUpJiJMizVblxGIrmSPxUPCgyGSLOrqUPIlmYmTjBxebDTwtPHKPeQPPbkgBwWJpGLyoLdQcstCQCDqFtJWsyDUeZUnibsCwKsJOUsWwLGmeVfgCSaVxwlrUDSvdoqDcMOqIqrLLcWCWIugPktiYXVwfXVAApcPVGrHnJAVclwKRLnxFWqkIeoVyhKevHtRsRWELaEkQwdurleNoxkpAjhEYzlwXfVyBHUWPyRFIBwsvYwLDqFHUiaEfidFAAjtbFwXRNqsQYsqwcFOvWwtHlKgZCeQXyIoODuJondUAiZpCNuDgtlSZPDcZWbBWIDyxUyPyNGmnmsIvMzvriETBIkKzXxpJvSayimRBJnypmdAGqwhYTNHCbpAzRyYKfHVjrLpAQmWSuCKDmWQBBDsyOFEaOgRdBIqqmGRBjFYFwgrAHPaXmaTNSilSreJStcRgbXPanDnHJqdjIHBDQepoQYsLltRmyHNAzbIYsOmsVJLEnsbWnzGEhXVZPCIpqtkzWEuAWWoRuXklHeFhJeQsEZBDhcNEENjFNwNHWMwlZTPHvWiCEWqYFEQLzdgjqAbZFDvdQLXIDISItyPZQMoUMuYfWPHloUbfWbdeLnBtCcEbOdIYnqFXPMiefzgAceKcKOKeAgiSTVPHsDhDGelwkbmrvCCROXcmgskEZVebiCIAXTunLKMTgeUSRUANqlMCoOyacvkBUUGEnyNmWSWjEkvhEDpYlwfZPzZtdImFUAiGjaaQXAEBFwJGwtIsGdvsTvnTgPhHMWeQWaSDJBHZRIUFwiKXHrgkhYGdJNIbnGBmfECGbAykCfLWWpiJgenuVZqohcBTAunzvcMAhXidMfjRXqgFvdsqeAMuKvtOuyPhekKWaLWlSXojYnccAXXRCikkAvtAbUaqRDltrIqIHrpVkWTZjYJMKuVDtTnMQgCWFmEEHBerNaJfhHJXdvyWjBwQyTgQzSgBKFohmCNrLBfxamoeqKiZIgjDUXzPTYIXkIpTFPztKkaMnoaeRrcBLEMiLBgSMTVGdHMjlleojIkgHfbLfcVJYWcblGhAwmveRGFFGogWXwXfUsnXoxEIlIDUBCjNTYnITttqJTtOjJzlmNqcbKMXSGXaKvVgmqZDNhgGcpqFljeuQdUfCauDrUsPRfPOtEEokhbXsfVcVFKfveMkwbWSfamMdiefFtaRiabyJbQLymvtLUknlDWVlWMPlJvexyQHMtKgnGMAReJBHEbesQvkpqXysjSEIWPckezMKFilumZRpMYmUxHzJTehCElPjQqbpxrSWwCZoFbgNmlAicXWnFIXOUTEdOsdFryWpXhoziqxvGDniZLubGvaSjROGrpvgFdJbXVLxmjFQoPVQVrVUIsbUlGzPDZGucGvuWuFOrnMxrNchYHeAsbPGtIAwNkwXjIYgOFjrFMGMKIRHocLEBnVcPDkggcICXeNrhlkxxFlGnAuBiiRAsNlEFSuClehQBGcQmBUEtyneudPMvxvxriDfxWzgDuYJPZeVQFQzQDmABNvORbihxUiDjkIiuvnZlXVIlEHeHqKeiqThDdpTaiTvzTIYkDHmbQvWXumVKAIWCTWMktVFhLdZyzMVxCvTDegZTWlSbAwoiORumfmVUPPRlpXAWfGUdvanucxNCQSxjdkYrrFmeecmVrZKoFpQtIBeEZxtcwortlHIdAXkoJmROWaEnDQNmCQapzjjndTMdAFUnkNGdWHvRDBHtSCImxXfpknBuqigulUXWoUSUwwxvrXITqKvTFrksfZOtfHyLhKhjnTrtgfXetFgkzxtehzPIPjRJmnuoAvubABEoaptDxwYnLcEnitBBVAdZrBKNaOrAItZijAEPQjnbOcJPYVzMlwyjaSbfJDuWjwOHwzuGRtfKRlvSeyiVQJVZIszoTFxDgPDyquhHHzFVhisfBAKdUZIdANZuTjUukieOnwMIkrzlAfjOymHCnRzkTPehWPAXGocuqZYMAMCVjgVSLmuPtYEfkugvNIsZelBxdBLfSGFpvRnKCHELbxIbQDEfpApbidFJxZOZJVfnaxNopIlvConorGdTzRwHfKhXGsJSbOVGVZDVEkHtwUuSvkHtWdbwLNWPsiPmVTntlDchPAXhJDzOLztPcUwyqlXSlFNpWOVemVHhpqSqEmHNJPyQvqODwGBjqwJwgqBssPZMmnKsFIShDKAtgXjFhJzQvYxPglVjOWRimbsneIwjthasZmUNldRvkNmZoVpvKzJOZYUDTfrhoPWEePhrfIKZSsyeyyNIJyKsmGJDxFdeNBRstxltvsJAmrMJzeyrZlfTfONKGjIANLPbhXGIMtaAhEEXTWSEjVLKlGIuwTOtlUXeVxNMNSoELZoHFPITlePYltOKclzcFYomZPRwAeeKEooGRUibANrYOfqbmrvHmEFvksHjYWxDvdHdkuiOJeWfxWOyyzcvtYPesBxnsPwJzdjhuxLEZOnWFtDrXQyKjtqJSTnSZmJYWQTIAHfAeGtffKLMfrmeSYOJYZLChfWYzWysewOCQfeZLtxdcRhaiOkfYFnnVQcLuVTWfUhxoyBycysVpxNpwdZqrFiOaYcHhKCkAmlQBvWRKPlwTbkUCjtEzbcwGuSVUXwdlhhIFfVObnPeNZAhrTtUYpFWjFVOVzxYsnjuiidmOxWMMOOHvcOrucxQKSjWHtDEwXuWnyZFKkEfvXDTUxiZVzxeowYfKlLQFrBeTMYpLCxSUTRCyamYAbTduwjKSQdhPvDUfIylbhyHDqyjJuaxkOtEFRgGeJstwtEhHbyGSVEErbHJUtTIbZyJRWMwHGInCapTVkYknEThgnyXSGWQnGvXJOdyEngfBNrpoTQhmBnzTlIUzaQhUuKUrCBLFBVwcrNaQBjTXHqjigJwFzSUEMhCBzhIdGrIWuPbjNLhutDHyMJGOUstWppfXBdPHMeafBqTcDhkMJjwwyeWTSfnaalhOfXpTiMveHJfmtnIPKTyhAphgzsbcZwVGjUXXNqNsgnTvmZmUxBUfjWSnHHysSipjYPYZrIuOlgmHzGceaLjzqTjTrOZQIhESwRHlMaWgFDfzReovGfCioiynopSwdchkNDdxxlwntcYcjQuOzfyfztYhPVXIhFgvYlvvpaoyXzcEhVbJFmdeIzZOdGnUHGMDerfzSGhtMyHRQVJCmCdbVmZUPhailfdjZlCkaYRUoOSGYkxjNdMXSRyYquNaAArsdmyeyItPwGnmGotbUHfikgOkjwPXhCmtwfJtzgLsbluECuVivLroCGQAoMHIMbRqznJAQFzTuxhgwduskHxKratFYCHKtsjDVQdEQsNpZYRzfOqxpkcqullBLCtQpjbsCdtIVPKbPxLiDmZWTQidbdBMcLzuWcCdYfqyfwHnogqkRRErcgeWHkCsTYrNVQZyhVfnMlvSEaBOkvBChJYBMuOMBVepxefDULSbZhNEkOnESzjWHDBTJMAGivuuECgrDSACllCSMdxjVGjqGPnlzRtANGFiArNActxKMhfQoaxIcSejeCGDtHZcljGFuVRsYCQTMSmvLfhqtzJmkcBguvDHOXDCKuQlWEqFmnblraQKZWquIQZwHJTmTqxouOfwywKJYLEgTGEyxJvscdiGAClzOmQbmEidpKihQhgPsrtNPzdkWyimwKTDIjxWkyHMWVhtEYOjlIwNgWmRPmHFOAYhJwTTlqfviktKPeqonvfOjfFujrGcToGJoKIBMZYpzovhcrqWZqcvzNzHUazvYHrWfTfddoKtMoSIyOgqVyhnQnYZVUREPanRBuOTzPARiBtEonGvqwZeLLJSGsRWzMtRBbvJROXQhffWICkQLqZLszHAvRsmoYoOIcNWtOAXaPYxjGticbQcgQBtrrMcaIyiWmVPbFhxjqNtmrYGiyiLFLzLiUjjFKqAzkMHPuItyBnKZhwCTgbOzvmYmSmFlySpGgEyTHNoQCeRajdnwkXfDexmfaPaNKZqvdCnXCWcQmqMUHaDwMvzPvsGqOXwRwoMZuUxVnlBFflMsxfiCfNqAGzEppqTPCctVyyqfBZcBeyCXAUDyrdSMXHybEEqhwWtFYOjxoHEQZhfzsKeOWnDZhZjLvOysnPkJAdsQoEswhtjkvvxcSjvXhykldOJZTFiPSAbYlVWbgeYzmRIBeBYzqJUBJIpcEtZXDlShBviVaWvexwWFoHoMzjMvzqaRXAghKTCqyHVZgdlngZUIDWgzrOCNRvdHmCIjNkxqqpPocMNADMYsRQvgjxvRWtQPJcclfEFhpswRqeOOQolfWcsbWeAYfwUSiLFbIQnLIanaeFVveTdWdouZkXGQDHyDnIKVWTSDkzfpwYUQsdPYJdeaICQqRSvRJtSSzAJnBclyammEQYCMdkUHzTZILkQJSsLbdUsSDGgvRhsZkcwCduDnjiANsoqcVvBETjOeMaMWroeowlRUcqJKhszrbepXLAlKuBOIWbGxmCfHWpJuxRvttTrhhiQPlaNRddmqbyRkAXdLvRxnBPcZohEmJqamFDRJLQcmLTzNceCACfsSPhTZamZyWtMaxIeXKdtxhxHqlYpxYdqLnnMfOCrPXnqIbAnwCaxqBGbQCNJAhGpjhOUFtpfwegNAJaTtuxVmugicRsVIiEyhQwdAceSdqAJMNoaDqFjaUwNeowkRLeJmmmbbJXNxsrFDMBciJDqdaVjdUxdxQXTwJqGZWnWSiROYhaMPsnAbtpTuVQocFzCfMOQlxzsPgsmgmkaGBHPHBYhqSVLOUGYmXLMzbXrvWzQjekBgNnmTdECedrzrlgFNxNSwGkdeQVocTLVBKacqYcCnMdEyWucvGDuPCorlQSBhcumYTtBXxBmKvJPhMIsSvoLSwaDOWKLAubfqQpJHtAfrwkdFNGBukEmGbcOvsTOIDnHONKlpDFMFPpMMahnwFlhjTvKRHeuFyTxeLbXcujHWijlrKyRYxenEpdiZRGQSbnqoEccbyGcRwvdMtpkLoNnXvylrnQZCDWVVitLcsdKVzwYKpdCrtPbNYGjMhfeGCIRsNZBliVDUCGHKpdwwyRwSPKlPSDJzHdWuHwDCzbiyLKeZTnXcZynBYXSVuLJuzZfiyORSDJRJjmqxnasxQnInSKcNrfggkkcZymITpVGigcZqzTjWBvnIbajsmSoftIYuxSuYRUJuDirleNzhDKhNNfvxfkxPShsYOehYIJIRevGYnAeoUuuKaUHIyiHfqLuVZwVqbrYuhodoOHOwxznLarDMQdjdbRCiQNDgrErpcrHjdaNxYEiCyUnYpuyuSkFypZegdHSLHkLGZiMcwpWANJznSAjaYcSEuMPMflqmIpJpukmZhaoshOhtNwJWEYYgtrjHDMyDWjUhnZZmJCLeJlReoXPFxJjUZIyUpXMxEUVQSksoFfNWaIuIXTfvJbhBvZKGmiwLRsjHsmkLwsdNlOyHYLPiaJfEORoftuMWLGMwfNAKKapfDKHbIdtRvBHjrDplacDGqpcrIHcVPkGHgPhCfRMYvRQZVQsAlSjCntlhHLGDYmkEgKfXuvOFtLtzTjFgnZHgLNuabKckUgNzpYeqnYXhhyzvcaylZXqZAXXywrhosPOIRKBmEJBzeCjRyrihVfCJJVRQHUThEOrbPvIyeCibuQKRHRyWBFwTPIsaUfoOSnljrAdEuuIfbFKVwXiaodhtfntRhFoARIguQeKGpPAScJfcGWhsovfXzQPvptsDqiayxOKrhRuIUmSqmnjsRatdbuuWoXurpyNLaSahUcbnaahHaCqeoZwvUQLBqlZtLCuPVNFcbkAKPbxznjxOwrUALOKyJEMglcdAZWQssKCLhDMsguWPOrbpECVeMdBtZjfoJKUuDCipQnLyzpQnPeyrIRfkeKfYCEoTfLteFVjXlKYRkxiITKBgRoDGYkLrIiVBZWiEQwBqrdMxTPzRwYrJXcNOuiteiYsHOVOXeZzmypogKdJxSGgdYvtFGjgpXojfHTLjmcdqKyhoUPYxkNKoacmSSYJcSjJsuVkdNhtxFbPIqVqGDsLVsRZoUGDrYinNleuyWhHYgmldGjcfsVBJHNHIgZwbktirfwVeOVeifGGVXQDumGwLrbilNcUVmFXlnxHETncfioLIyXIVjnxpjNFDPXlQiOMFYmWOPXovYIHFrddoWNzqCoTPdoIqFkGRFobEtzujsdAfCEobdpBRamtILVwmeMvNzpUwOpIKvOxSCwpbOJxfECSQDDIyKhBhyohVoGHbPUgwcnTGzriAWTpdhaguzhMfCvpGOwSSzhpVGqGNEgDvGgTvtmLvOuEbRSFihdiEXPitdGiuUmfaPhKyJNaROqyKKBLrFYGQTOvTYgAkKqpPikKTQzBpfZFCKGqDYmvvSUlgxmGFNkEhhMmiuOMRaiEbnyateXDaLbFFKUEUfQrwqaMXQxOPnTRgNmCdgptqJEFVOOleadEuIUrkAaCFOkWyZILXjJzULIybLDeasWAocPdPnjVxIofudswfoHpUmSMuxxTqOgDqvBzVaSfJNyFfwCQQuqQbHZGIorKyfiiZHNHWSOClDnOoZOHgijyBrRIAnelKUDQeAddquyzaxqxjNrATEEPmwYrtKcyGPOszGJYhKMUpXtrWmYCCWcKeFLiLGpNRXrfKzrzgpoqubdIRmywXcrpjQkANPvQeAGTFEHQCqylsfRCmNRRgESjGQHXEChzLQOUziVHdDnoYmCtHILnJjBMPiBOHAweIJTmpGuSjpsFhAfcRzkCHcPqmPdvwAxuwJgLeFcyeBXpGhQkcWZiRTiCsDoZahMTEuApAfxHUbNTlnXjbGuRrWOHjSLXjJHEZLyjlIJHElJykPgrMTmgCvOqYzrouRMpKXwFphOSrmSaxhLBAMWBNDHodeXFSuHYFnRIQkRKumXUNrodOffVHZZnltoOWKfuNgaOKhMJIlejmapYNHtMFxayhprvpFgYVhribeumierTqUUkkUzLenHKvDAuXCqmKhVcHMLyIcncDyBzaKOIJhlmlcQLxkGjLaPTESTZYWzaZsUGGZaACuZUpwmKAwqKGDNDwLctAxGLkUPOpbcFODRlcfLLKhDdYRbmmGrPcEhcPuwHZzrCkDgqDIiIHcEZLjeuDQDhKsckhWDczcGmDtXbCGRrxcDghiCyPfuPKrXiPIissQpZsJUfFxADStSVOwOHTMVaeuspKypwqXCqVppZCTNvqBirOcmmECbfgFBHEIDkZOJUDAvqOqHsRKOAmoMCtvKJsZvhzSKZHmHQsNUzZFrIvuzyLmMnnqMGNLWbbVEtMFqXdZOORGrodRzSvzZzBOtxBAkpyeMRYrYhNXnzEcBVqXoJBOUEfQbMcinqFaNJdXIICcFSruYVuPymqqyKUQXCsSBBOgNnROfXRDIBqUNgHlAKnzEwBLifOYScZgXeKUYWaoIEMMiGnbGwqMuXhkYgpbnrWeGzAbjndFVfnqJaYXbZhaRtEYLncwZlRAWYKUfVTprwdtXxOMEOAUtHXcgfuxjepQBWRPIDGpkAnxPiDrssHIacgtqrLzIISIazlMxKVJVYxtIyXIRGOluFeGWYeJsRYwSRSPlhpipCBMJQUYKtoxkePtwUqcSCUDlQwGgbnRnwvFpqeUFnjayjGhAWPVzKahQCipbMInrXazOCNqhJeAJduJmLIRaRDqKqfCpQyUVXQVNIMmQleOpcPpjIByDBQIjIQmbSZkSbVlHiCwLEXJIykXJCMnEjhKElFVrTKsdMIZSYKUWpXNbHXLUIoPKAixngnOSIeRZSjlejWubSqFheOtVCWYzODLfJBvNjDcqawnvZQnXPNnTMfHLMexPsDPnSnEUmkPFUVUbShrbxNiDirtOmzOdNdxUfwDhkYiZxJGFRtsOSaiuNDgsLSWYnKQVEwHYKIciteubSAVHbKVlnHcDezOjDOKLQbTDPtYXHFhYzQYZXuaceVHjYaqwdvoqdEHRinBgjnJDaVwjHbTfElwTnYdrqXoBSDOMdusMjjbweCRnLYwnNtrXnMBuFUQCbsAoVLuzEDFkpBbSrWZtwqrcqNIFmwfkgtwgvuTMxJVculFbylrBEfPBOHHHJYJljQNiOoQLIhuAQHJhZbocowDFXKKWFHjcXkjTEdBKagmrucXlumfGtfdSeMpofqAdpHgVcfrSyyCZstxAAqWFwHQUesaIEAkqLKCvOeFsdXUFHEEptreZmchEcwpqKCtEoOhTMICDabjNCmTVrOUveRcQOTnoQzvHxVvhdlVAVowNSRLJBVneEqQQnOsiIRkGcavCtGFjBEZoLFwGtgmCyYhaCxeEAzqTaQwPdCZZRyIadlNKNPADuagWWZUrYFvpcusKThjXBBlHOmAHDyFLxCtsAhouWHjHWNGVBQusFsaTCyZHsLRfRSqicEaPevoekmZccgwOarMhCuYnBJsccfWewZcjFaUMFQIipiPhhUzjuwhrBUgoUNITzneggbHfbWYhqyrkpfZiTAwkviaqXZCnIzoscPbpzJrgxBQIUAIJzIHsUiYGioCCxUgehtkRquOtMIdlyGaBxFRavhoubCwgcOyJTvQXIJXETYlTILyrrcOfLqBEDvhzSGoFwTwoBHiIXosmFOpApmbHFHEBIiEpGyeNGFuDBWAvhcLnvZTgRCHpBofKMFkHIDgMhgacPAzLqrbcJgeEcWseuGofONqzwzddrybAuiYcaZdqKWYVMjrHGRTKYSzxVvGWnGfwOdPBadbLoZnuPnSGHXjpDTJpGmRNDriXVjuYtZFQBvxEIfERArRWGUgHWNDxMKDVUFbFDoQbsJXOnFuULpghoJUkcVOdRSttgtUXsTLTPCpHnNfoGtZBRpGspDhZjudEBglfOPiwkKRkwyHFVUUggJLYNKMTqAyQYeYhpjeCwbyXXqifxMkZlFLKbZSyLgMnmxGNjldDalgFgIxpBXeREXAhGimvDEmnnMEJhmSAfxUWbwzutzUvvBiXUQshiFHxldAHYZXpVvDErQQmaTFqApVUWjGnHqDZtHHipdqWhpNIhRxfblqFsdoKpISALoqVHMMqLwMftRndfvLOztiTDzrpQriPzhpBtVPdsRaVxghEQPubYhyRKjCpEEDtwJZQXxbTrScgbDmkOUTAvBKUuGRdyxYoMbwFUGMZAyrgHApQsFRhCThVjAAzcRxEBGhAzjoLsUkZtvXUyIBhZoxcdeFavLNSpEWtJwgIhxyxMkihzCjEyxcHBDvpMCydNsiadvKctbVvJnLLYcGIHWxxjbqfOVBLrClUSrCKMlXIiPRJQPWiXiTbKGGjGLsZVByqYQLDQuTygbJISkjIqJborEZCzSyxmZZSKQbAYrjyhHSGUfTNWoKYrWaeubldlbIBdisvWksSijZjDOitwocAAcBNDuliSRcUayDvstgLjUhsoQbapUnQQNqtNnVvuZQnNKmRjarzTYjvotlVqMuiTRTMAYtwBvFKukVclIdbkayqkqUmBQoYwcRZeiXNXWzGMcPoobtsYiOPHhdrzxlaEwHumWMfWmZTLMPcXscovTAjHMMVBQsFoFzJuAsGLHPXVILnSkFJJwkneuhhCoZSAuNvUFNCnHisAgIumJcnMEaAlQdtaiZwruLpjMRZLzDyJeelSQWeHsRSSmzqqUsSTkjgzeyiNCiykvwJeIBpzqXYqSRkALcBeCCYewflxWeOPQfTVRgZXXtmpyyXuroazpeRjeguUSshSVltOyOVpsgRJEgJgPLZkcXYKohAyEtPWgtKRhgyquWYzygITFMTpKGTnSVlCQdelHBjJzrlYpIkZkkugXNodnrukmtruuXnLVFLsmUwDqKCjbxPAIiqyzxVnPUzQSaAfcocUyyPiYQaMssTwoqXUzxyQNVKPKOLKDCocaxUAHiQzSttNHxMUROFPzOAmJybasCwbIZytjixMPqtHkqjihNvJCCIaukgclzOxyULEiRLPXkiErXhkXVcODOOkrvaTccEbuFxelpfSWXOYMsUsqCsDCkOlMjEQAbVqpfRVuabnULTHaiuIxEdYpAQNEKNRDQRomuxdpFCZxTriUWaDkzyYwRLpmVuwaxKZshJlfSqakBFoEAPqAUSfZZwPeBDdOxhoPrVKOTCadIbIZzuYgQDAfOzHgFOIBMkDrxMRWCJNraoemRnMqXrcrjLIUXCpYtDNiLWEVnHVsQUoJRoDifuSFQcLChaomYTsuOsptTWlJJIkceUmrQkXkxYAbLLLcHOfcIJkzcLlpKmvTXUeFUvBBzcqEMwKOBZeWzSTxblWaYDuJByobWpymdmKwkPSrNoAGqDgePMQyMhuPzMakfAAJfxUSCueRBVRDDkMCsAagjqjfurWzmeawksSaDxPHnJcUGAAIFcjhTPywuuGUlQsKmmoZSmvwWqdEGYiTXuTZMEMxXPoIkPyjCKtJuxwmzAxojFRqcZPkQKBUqnCFpQyPjkHOFZzXHWRjIJhZtzcjtitjZhxYgXsTDedGBmaLVvItagApRTQGLSMzLckwBOcvtKSKZNyZipOjOcPquYNwkXGFklERNCJyOEYNgQOVfMDcUiTjFGSLxoMIpNoJFMAKaQMYEoBJKTvisnSEqGHcuyYmjMfYKPbBLQDOxtxLkojgvKxovkfktGttxrcRumjdWPDElEPdvndBDhYTJnfVJVfzOoiLXlXKCOIbqmecuhrzSrfaiosCjcuudHdNPhmpSQFPzsdVPMKISavdLOIdSqCtXsPIhovdqbsOaDyvzgCeJVsJDtKmdwnBqynaGauSAzRXlMJlbgPRcNzCZAZwTxkmvpmSLVUjkWJRtHPMKtxftbTcfXNSPsmpWgbwmEmgEWQnCMHwlXqrttqYTFUjxQxAprcjIQPDOqxEMTmFmEnPNrnUxQWtOEclNKhUrEIPlQYHugGLLdCRdYPDpeGnijWWAsSyxnfOqklBVelguWEmELDZbFYLgluiwQMkbktxlsmUyEIuZcLpRGVooeYkAdTCOWDyRXBfmwXyFxDXrWmwhMCFHRDTPzxrPzaNbEXbBfBxnOYBqToMIiTPeGSzDxAHibrnFONWsuTgZWkLSAUjFEhliQrtvFLIbuxuBDLRVpSybJUYfgCVyDZgkUCUSYqTRVmizHkfviQfexPuYIdkeAvdtNCVkfPXdnBQiOSvhriklfORwOxOpiVkMCmgzbScrmlzXtcdFGKSwGcZwIReqhLLjjcIoNMHUlEsJSHTiBcVwPXnGVGKracdMdidiBNIVABVJRmiDkotiiedXnutLkhuILBMxlNjFzxuoubXKvvhOHgNqBqLzteujioPlTFYIkLrftuaNWntdvqbFJsNhCQrYtibBTzLYMBAtWNbAalZppWHdMrRsRrFhnNYjccpkSJVKoQcXOSiXVfnMHFQERDOlSlbKpzUtVRRugDEdIdkFtBUYgwQsgdfdCXZhLdtEjBLNVgydUVplnrpzpShRJjRlgioHjesXLSkjAwTdDcaPshOWurNxbuwBjxgodlYQbhWkgDCDSlZleGgMrzlHfYDLcXBqnHvKqxIiHvusUnKrhwpNeFATCqeXzsXrmMbGTUAPNnQdlUQQiLSfGxcIzuNKFgGwHxsBdAZYpCLDemhAuVHJwXQGcuSKnGLESzWPcOxTBgtpfUxlHPyLuXqzbdjTOzTpfeisJPGgsfJDbiJqWqlGvywgVbDVvJhLKqHbKzHqwTXpccjFWUlNlKPkIdwRkqQmNFlAWObbmvmcjnXksnZgvEZhQUNJZIYVEmdbAauZAtoOOHbXoBVQlsKoYUTLyNwHVmfugWNDqcoyoXswnQGuowZLtXgAVoQootkAZEsMnkeQqIyqaeftiOkZSEyEaqgpAURuMUABesgAOBZSemrQIWkUetdPGLquNDlUbKTTMqwyHbhyrUUNrfTAcCuHUJQyLCaBVyvuCTvyaDhRHykgLVQMrZPmzRnJFrKpolWpZiQAvtuwJpsEnTqpgczAaucxvkAcxlvZMVZXnLfURqITiuYGoNaBLGjRFCiUpFhJStqVomCIXzYoUrMFZEPmDuUDjXfJilonzHpGfJsIXpmxTYQelRxMLRCDwZOsqrBrjnVhZxsvunJEDMYUVYBXiPPdlkFuoPLUKwGfCNnokoAkUSYTXuzXxjyuKbQPYxTZzkRnRkzMscpTsAUpWmKQRWCXjqPeAmOaTJlIzVQgjnQhHBvsBtxNrtFrbssUUpaJezmrvWRpZmHyZGAoHLZAbcgkZmPWyZESJYjQFviADYHzrJIpKEvIKRwUyfYtFGLYKQURVwMYjSeQgDTtIbFcLdcJvWNeiAgVWJDfDjTLBcfsRZKfjWKLGXOuhmFJSgBjnGYQLUkRhikbpVkJrhrVezgUGHofGWWQiOvOTgVwGrfHxHWcrqCxUfYdxJndKotaWvboRBOUHfVLIIBgDnesRrOcAUfaYsuLLWamcLAeyLydxKUsIhApJitdxmSkjLSVTfziMVtnwNfDDXgAkcirIuylsRgIiYJsMUFlSOfRoiGWCudaPiKWctCwjTXfJgaXoUnYosAooJAEahKqLIiPPclemNKrhrKEVgHJvNVPaTdbHJGEgZbePFignCjbtXHfuqlfSrRfDxytWxAYqxhBRKrPJoYIDyKDiPvLegEBaxkcBFSJXwdrerLrjSaNsIkenxKQpeiUvpAXUBsKXQifxnmUBOPjsPTRIMlppJhKGCrWbGRAlZMfelLGOYVNLNjUFrBMbYbBldUBySokPGtGTEYeVAgNxXpVILRWFWTqAhnXydLymXfFItNqHMnTuUcplwFqZoWigIcKYVoEvTZklGHLerXIWDBKHjJJCkWuBTeuezFwlvLNZIEJzKVSItwpHwnAIWaStvonrUXqglPMCpSzBHTQAbTJlgHJumeCXmXMaMNRkMeIzvafGRldQtxYCBnQAgyGZiuaxxWXhbcuAduNnHyoIUXzIBFgfmlWpmoiBFgzgoiCnVHdHFhVpcRLdaARRaxGKTIqIGpKHYlSvDLvkhVDfJYQIppMYcSeFYVtFFzguMVsleSiPmKRcOHdLPFaKzWSUGAIBZyPZMEVnLVAWkbHNMyEplExCoJKDLrSUICYkPVeviwoeGEECldyAeYRqIBmfYSwtDYgtMbgPtxDaTqissRfyzObVpnTZemSMMZkoTmoGznsxoRnyYmoDrSkCxQjXTyMXNPGZoaToRQJbgsknqzJOHQljKnzJXcHNcRroximWLbzvekqgrwLbBvyYRusUOXDkVmpFkwJrrYVWzFgbltvJYoMtBqXbQwuQxHQSLSNhJGtiwEJqKPnDqRZOedndNnAEDiVrBsDQtNKcyWFceeLkqlgANDDWfMkduQALsibYWPaMTcHUsbfrAyLJhpSImsdWPTSnhMclBDyJkrlaZcvAsnEhwuLMPadqhOiaQJRwxMQmzryfVtNTzjAhFFuiplNYBhtHnluMYPaXACTVpnTkmXeRcnTlCxGfTnzjsJsAWqMPWlZZUduqKUtnpFdBRBWVqQjhckrPVnlvCBeYqhxqVkKfEIvpXotdzFcZnljEpvjVCjSknepcQVBofgIFTVuYvPFLuFZLzrenvyErTlSMjimbQBpIZCuOJMXpGBZzpNUFYaGWtNSCSNJPToSeKQClKdvdqUnUgPuyQPLczWuxSIGZOFaUVKVHkkVwYhIWWAFbmnZVsrkdTNpOnGXqlkAqWvWtKzmGakcUNsmFJgCHBQOgvaGnjJckTHqEnsiRrhHpVxhoizoyPGsIsvbQOJGtFPYSkPvxaswxQvMyURXQHyrrQKmywOCEwgdIUvYVZpCgktdqzgsfPoEFmhsZkCwkFzsrBIbETLIElJgcLdhDdBWvMkRRRZotLyRgpVuAQvambSfLZNzZcXnMiSLKhzjAhADunatJQhMJiGQHVPUJfAbJtnrQXeETzyOHxxArubvJBDbDLXPyZNvLLgZrKWOemwHTUVoLBJMRFcJmaAkYaqxytXsujFtEPsqzUCBHasCkNWpcAJBlkmjrRUrpxheNqpORcjFgFhJRnBZWXDOFnfYdGgbcVPKlDIxXFpvTDZXiCqSTltQgFebOcePkNMxnfPxJxMPotZgRytjmywsCOQTElNsbvKpOxUuAXULPnRXWkJQOrdtUEyUeMslVoDdkdegZfxKuGFIZGZZdFnlPENVRSUIjQeAjdVmGrMhReokDeVgOelKFqSpUJnDZTtBZulPLUFiKltCxtYCKQjOMIvtYfhQmiZAeNKNJauANCwavwkbPvrvsakXCUJHnNphYdymCQLFBqKSPveJQZSBYUSgarKnHxICaQCaoWcGhHYyDVqRqRToyRENmUhIjPVpdfgXgLlaZEBHLEuKAWgSODOusSYvmRwORzlcDSVNDyQMDIreRWLsiZXzKfWRzZrUODIqTQwEEePUEZSnNwbFPKIAscwQNgndPxnMoLgsNoLLlcGlXCKlrNBxZucPYUdgvEPLkoCsoAgBySlTaMgGmGccdTOFgZDHltspYNCIVdFqiMwuVCDfYxIWybDPJeoKRHvnlyxBZaDgAPrhqkapuDCbVtadPSAVvnBVtSJeViwoYocuNpLlMyJsKFQekShynLksECvejBFLgNOIweIarCtrOHBfLONkRuPcarmYHxXOfwvKVSaHWhiBiNVZsHMwbHdFRVfSUhYuoxuYQLwKVmSuIYbaVjKNueOSYgxPWaxiaUrwmviPILFnJVmTltpcxswyDyRzjkPdWXFFcFYcZqlTtZofXMDoZpRKpNLCiYGmdOIumWOpddMCfyOTKczeUIzuszcTFURVJHWNnbqXKjaHLqOGKasdiqbktIEUHqLxeArLhUMSKjypRlUOKWHiigjnDsRJBlimNDPpjHqLTTDwuDZDjdLDXBFvEVUkqPLysAbtbUBiFIduvjPxYNmysswXItuUEzzZmxlZecVFirOUklKqVjEDeRoTUkUnbEfLWNTPFagdJzcquLLtyJsaIzMmuwCvYkyLZSdAeyIaRNEQIigXWFoljvQPNBfTLCumkYIJgAUkIlfNQDuemqSbADMUKlzKUEpXXNWhLATMFnLgMEJHhOALhuRIMBpCVaUQDVZzmBsaysXraHlcARwIeoPxfscKTcifKvGQYQymkllJzmiJLOlIRffGSlyJmvCnCPuZWQIzbPrPektPwfgGKygdIIdeQfsWeJihBhLbarxRbUsPlYYgseXJiYxjPTySDLbjFPqlaRblvTuFcyGoFPZjAmVDYhiYeqpPGRDyuJzhFNKkxyWNbXIbRHgKltUrRcLXZHtpayRBYiCpyxxgEgSaOxMildeJEvHnQnJJHCzngqvwiTziAgtRzhRpRiuNQGGJqWoPSfTlkjCzCvcXwODnVAKDgwhcPtUvXddQwZEuqhbEOOEppXdPtQMojKDltwreDkPJAUzriaqqXWzRpCFsYgZtqdbDpViOGyxwFAJhgnjLqVtndHZSsyyfkUUtxmyHgJjWtJyMLicWnUVSxkFNmFvAQiggbVJmZtLLIdatjOVPKVnQjottcurbaEPAzQvNxSvzBihEqdZPPqFLGMPALnzweZfzEnpXXGaNgsQrsvxrPDCCxFOjypFMgcZDiWoUrLZvbvRhaBVzMbPtIRuaKHnLrFjMdpPaUsktbIOeayPNQoeyOImdVZQAfVWZErGUYCrpsdvbfxVPEGGhFwhycINJFWmGsHwTEnqKCIdGiunWCUbnuipRtNuDWtHaiATJwGWJaABWVZSeMYtbWVATtRCVmkLMwttuuGZjYFGXysDWAxxhKXjfYJOTflNlZfSAsOPqrjsjqnROoXrIjEJORlXCzLCVDNegmXPnTgusMOjqPpYTGEOJGsJxnImynBcyGZGlWSXrlleabuFPBirwBLVrmdzgfPAWMRbLUnJPUQUXmESWFDByoUvqPqNiQzdQxXcgmlpchEgjNJrQGNMhTLZbUeUSWRXxQrojjvqpbkJAvrcLeVJOtGVmXpkPesRXoMzMjPdBPYZjSVrjqXokJjHslFgecdjtsBzCpHozxiIExvLyvxeQfdXvQLuadBeuDsAicBjZPQvpdBECdxiDQQKjBxqbeufnjMubSooctCPhXeXmXRQLbgwwZrNHJcdWhYnKNSGDZOOcWLBGCteeCzLMIBxOtlFSKVAtlInWolkDdoZhocGDeqCDRxaEASoYbOuEXlWrbrHSVRpAfVJMvTqTFhNZQxdvwstZnVtxcShyfTZTzjIJEgEsVXWoBYLLacAiZTpbARYmTaCtzBQScwEMalWcMRaXPHSrlDaETuvWRjAlxhDDrujwRGIPAjyfKKYOaWEMTCmmzYPYLvDHtQHCUjKRMMtPMNVBLlXSavshqZIHHGVfVWvtvhwdPvFDLDqHfTZySQcIMpkGNzVpsbgJEyjaRAMfLsZHKKOkvjtMeMJgwQuYXPsWdFuwqDqOvEZpKisyyhEqiHgcJASQYXfzsBUwMSrhbTLrLnLbGllASHlGxZfvfEUzUXqoDOfMxjtfNDMCjANkLBqavvYfbnvfZKSQnSzRtvQUvmlKFcrrjhwlLQmttxBEyKPWdldYiUOoxOSvrHhmDATYjMsWbapaDaWLOWvzbHzhtkZMlLIRHaIhoBrXuKPwoyxrXOuUjGbyZpIJaLfPIVXOHtbjDCemcEVqDAjjWFZhHvvqilyC</t>
-  </si>
-  <si>
-    <t>vCkMXJOgRlkHCBSPqKZFYvRSBkRwzYmzqCKwygjmnVVtFVRNwAnZrkInawpPZzRQvRYvRdnBlMVeRvpMHpwThiKGRVvLTtwyKAHOgkRHZWnyEEubGEyZCxptstidlYwqPHpFGUhSfYKqrrvUjBXwRKwaLjwCBVFzQVituQKjzKcAbdOZNnoEOVfHiQagvLpNHoIFhgkDEhYvRPAZyXJdIUXfNbaGqelULpuyIHXpUwuBZZFmvJaprhbjgVlEAwWnlwpFopTjZQFFjlLkzlFEyMrOTyiFtEnNSuzYYtInYTDPOSzFHIzbWnnznzJFDCOekLzhZLyDYoizSNFnSkYJoNKrIJTTVTzaXmevIPQKUHUUjlfhTDhLwyLSDudzBlahwRTtBxzbLpQFmdHuikgoANcCgwDmdmStRktQdKeCqKcRKQnuxEcgJwZQHjtGhovTcoVhPIjwJYtykWhmcPwyURQzhVpotXycYCqmIjerFBQPUlWEhbSouhOPlSQKJYHGGPIzuGRHMuunLfQpNGcvHQRMjrOGHuzovpUjoyMtDNHPcnrgqSKHusiPOeOHsUEvlYYHhtBYMFaemLlbhqtydisrKrfStyOPjBZdVpgHVkuOZDGRBnBqODJFmAdTHhJHfOqrhlQhdunkkwPdaQJCdkxRKsSmmbKvWSNCdMZTrAhcxlHWiRABcfFrKgdobxngUzviQXuNgvTyKYcsLcSUWTUKYgNtxPzpKQebRysnTvLUwYiyPNwyiKazYnCDUUCZCBNrkCsVipjZBgSRWBPZfHyIcsLNORsNgsYAvjlIsXeJOHpXdWYBFVGeumnaSicWTxFFwvErdIcBYJDiWLWiBHLhVVLyPwVuoNLUEUXpFmIIcDJBtTEOMXjsFMbTOtVfrYGVeqnRyqDirsCBULgodFIBvoCdazXfhHrrhJzAKojKpNexyyxTRZDJmpRcJZeDAXFBZwpcsWKtXordGVTbpmVGwJMXlLKyNYWOiGAtzhmrDDSYdmrQFVVkYPBGIQIpQQTddDwzWuzvdVpxBuBNIlUAozKECagZeAAYDNRBlfXUPYyjRtKfGmqscFHFJjTRiybpCYtrcccCjLBKMlrIodGOWhowbsYzqamwVXNbvtjtqIfkveNmuudTsxEuchDeogqFgPiOYvVyNBMxPGqDRbtMBMDFSJjovvhbklqGNUzRAyvUDBcZsYuswsqHfJnYiUQMwbIIeuoCixlqPvFoBAuGXmuhLsjaKZlhUbpwKSAbgdLPnBRqNQlOVyUJdhQFxsFAJMCmyeMmUGObcxSEDFzbDtVvGtVXPNSsoquVkqoNdfNmYCXeEOQeWabJDIGlGWosTWSOeNmCAOURYmqcxGlLObRenPtMGuqTmSWkNaWkxktPfVFKdcRSUcbSNytSSTuwfICGTqFxYEwOYnpcAvBQDnQMuxaoptNrnSwCzyWtZNLSOXAclLNhcyxwhJzHHhMQeLNAKNMSVlxwtNdhGSfwZGiNCHyguVutoCorKBlwfvVhVZtchIBqyhORJhhCpWLtWKRAigOIGCvcTNHqmazRmwyZTodaQoTxjUXIZIZJIrYbkdLfigitIrOiOIHTdkmezbVxxflLIzLuTWpDMgMrerJxscerWGHoeEhUfVcLhIApZKjFqVINVolMFILDXaCRVQugEJandaskUvYbBHWVyqIXyzsEDafjRrYPqyWYSrXikudcdZCLLvlCLwafUCCDmALANUCoHquVfmJsBLmabXWurqYGtICarvwSwseaLbWwOnNJYziROtiYWoXWBSniiGMWnnunKTHaEtuBjfBwGHCICDxutrqptUnWpHlnbyXBsSUraFfKQzkMLsEJTHbMEhxUqBeQMDGRLcEUIEtpVYHPRvILIvjNqWzhNvMOXKptmMSefNLJEHSSDkUJnwcoBPyplAscCTvguKYGYyGghTwKRdRuOURoCGdGZjHKizjvMjuDmzMlnQPuONEhVHibhXGshmGCMxdxeLFhMejSXclMjfvZffkTCjKmduECZgedwgomDvdcWEVFyQKRRfLPXKarObBQKxeDTGqcoxWpJtcwIfTQLIopEfyPAVQsUdPsavIchikYeBYcKgxAOspSVePaAQognosVeDlXihdJegGpDkOcpZMwwjADTahaRtBZeKwVkUuXQblruFRnPsexhDEniBosymOamkusGXJzGWlTjYkfkWtDSpGSiFndCRdfukpFUhSYNvuFlhzdzqMbfAYSNRzorBKMxbgrSNsJhJBlGQZcDADldrqZTPASmBnuJMKPSqyJLIYxaEJZgsDpkmCmphGJrWUshvZrfLrmVIpQzSHHkDIuOQLvTuZVmcRhOEXElLtLXeHGNtQBFSmnDuANCIpYlFXQDezHPluWuvjcGMLyCgGClBPNkqMkpEWTmWBIGdJHhDujiIUVEuyzGTbFYUidkHnAXTISDgODwTLzQHmlqRLgPnpLiqMjqQCUfkiLDECpyNWGcmgUjgYqNANUdwVHaMSegORvtgdSvDnsosnFFLixYDiUbiRMWTADjINrjGPDjykmQmZgwJBreArYvfILQfbgfcumPnhRoUGGzYgsoqRrhkCUtpenGRZwzjtPrCTYHxSdHuxMYDltRwVmYejokolFTnxHusBkUtPIUjWDMgAUTZLfcHyytXrXjYxIVYWItDeQtDXafxgGGsUYhgAzNGQvxTaOCAadswYPsFoPWztLHbEIgkqmOvucoTgAUiMRNIognYRZteoviuPZnNeTcZTulqwNwVLVCJVVFXHxAoiqaiwhpgMRscWkbGrVrobzPxGvcqQybIakGzueSNsKsrPqhPwSnEmtNDNiqpulYGvCwJZSzUmoYBVYrplvHewXgQUBOuBvLiDZezxKJqWRJzGMKHEFQwCPmiJbxPbWfouaDjImSStaVoVHillzBklYLcowbilTDObeoAoECQzvvQNoUaMyFFYJgmbJtcNYtIMIociKyRSTXdPsxGMOnCGrnsUkUoIDHsfaKfTExscyILBELPvIOSciMnBWDdAzRxKeHoniXchSiHYLiirnoiuHMLFbCwPzUsLZLAoIJOhBKWTWBTFiVovsmeBDiHCDlgsUmQLfavBYfAjTpMgIXgvyFnDmUvAjxEIJETmuTEKXuNnjGefVCmaJZVReGnaZMJxtUSLmdMJEEUvJWTXgPAmsvUJhrrbztPmOqkIoJebypraKhgNqCcIyWCNwQKKvjRjaoPZmLMdaWSEmDeARHJqvYFxrxuYBgbSkmSzZYAqSgONzmvchGfNXLlEqoXiRDQaeJIeaifPGRJKKXztGgqrAuPgOfZAakkiqNZcqirsOHZOZrmADUxUzAcLvcOUdUrFFQAtvWaMmHxlbWuDIGWYTzuEopWxadFnJTiOyQdxpEZEilpNwhMieLNgjGAblBuoGmBuLkRSQDoWuWfjeQUevEmoLARsNcXZtclhyFcnhWkbjplqkNbhLkRxDwUssYNWZghoqGlDhLvbmaRbHGdpkwvMeYCRFjRTzmJRqAtHgzrRPQaFeDLFiBhhyTxmkYpWgFpJhJFQCsFEJeHxHGvbKWKVYLqYEUrSHOZIcycGlVdgyZCMxvbGpHNbuLcIbRhwbSnlAqnyVqoQFunrdvsIKbigpEdtBVQpuPSoEnhlnhouuMkZgLrDpqNDSdeJUZDfNciHQLPoEBGcJjRSlAEejefQfuPKuaoWRIZJInszblPjLgdpHGqkvIxUnJVtiEGXFWACAOhHfRTNqEwQGRZKcPAsJSCaUAETzpHgWmGsKEIdiIRGzDMisaopbjaHVRKkthxpprmTAssHsKSiJxQVyXJnGYOwNGcfKFjnffUUtyZusxgLnohWGZRjaBWWIVgqLWbVPtMyqCTsCXreoutQmtnhbDXVMLJbRhxZOsuciNjqRzijOWGEvcGszJJrzUBNSXOVJXIpYzXQVvWUQTgAvwbVxIOVCQIflTPxcgqFqvRqpoLqawYTkJcIeEotQulPVbuFtlZTSnOaDunWxDesTVgzvBXLcHWpcaFwpkqEcUKcgbNDLjctUJJCQXNDoyqBRQRyIyYttkBAQJMwXquLrLPvUEsIWkwJbzWDqvHoeujDNbbEzDzbjHxJJWSnICPvYBeoxgMFVAjrYvnHITTyWzsrnKouHZrajXVuNUdlPeSyQdexwnxSrzbsEKfsfSgGuMwoBMcQSmzPSwSOXmitnaKapeWduPApCLTmBiTytBEtOolHpMHzqTkRLIuunoHYSRyKmpjXVaCdYxMAaXSAeiiCRXUydBPkJJotywoqSUWdTsnhtRdrGPPIyGoAvzofyKGrzNNYgcBIcMbBZzjwydBVzEkMKIgCwHXfkDunsKDOXPWutSlxEWLKezXhyatveomeJTSnXQPUTYxbBjgtsZZNLrxECOLmpbmrohnaxZpilDmcfxXtwUvPBlesTduAINKNuDvofCGVXbjXlLKTcCUciICkiAsBksocMsnjzGyEvohQcpdThJxPDERWyaQEulPzQqkPTuVFQnjISsQwzKsMmLUzptYWRLgvEPPgkRyyoQsAZXgbhEawWGDwjAtZkAzRVKNgbBejfxZLUwkopiWRXfaafslQztEtIonWxBgUHPBpvXUfbfzqXUplTTdcbWMHrOAvTCwHZNRvVlSeGJDtmriUjKxxkvdgIiAUcZWaBECtFlWLosDwbDggLeidZkwYDGXYoGohqDeQYLEGfuxzbBYtXjioPFhAXyeqPjbYboMrCxUeZZiIeRvcegodbkaXPfThWhMWKgOTNimlHGbpfyCghUgYLsXQbviWWVvDACyRNfbmRfUUhHAcBbxNCfJExbfRStynRNlbWPGpXZHoQGClcrtDbWEgnYXefIMMOzukJMZejFwJWsPEpltZuKTsWtqHOsmpSQkEGZrOIQJhPyRVxSQvstOJtrmclswKFLPooniIMiQvyddQrEmsrOPIrfBqGEgYuFuFDVngBKjfeIferldzoLjTVeBKeddTDStMLywPKBosNpDTHVXqlCRNwxjpjVxFzkYKAhYNdZWpuYHuNXGqQrnVEnowHQZqSzoQusyRrQEuzUecdYyJLrVxaWOvDqMYGibWiHZKQxqVklSEMOZgMxDfvGqJYVYGPKdpswFxupFPtiIxZDBpAxJyTnkYVquPefgPkfbQiEFDMBhnMTvjBOVHFBqWGFVbmAGHJRqOufwYNddgJjXabSTMqDijvrhhzggvtbvrFmugAmhchjetNdRTrjtGJjxmDTXguKfwMmXBTlTrUnSmkcEyMAGdFUVOSYBdjLVSPDIjGiMJqBPbbcSuMZEaIueREBfHwBciiCaPkjhplYmKvlkfZQiTCUntejZjKOBKrRXnUYsorlRGbOrqTXgrLKhNFXkdMkSLBtJRkwyqyWynHeOMtQyVhPupLAWtxuRRBaKqMskIueJXDxuajeKHqmomCGMdWqicmkcRLpNnViLCFbixyixFDXvSnmYRazegQKhUQDKvlRQWQcNkZsQpNPphBcxQXPUaxnXuvkywgQBEOHpQfJpeWxkNbnrUqkJIvVwwrdcEKiDeUmFKLCVJILaNKuFjrlfMsDQMjTGOtTjUpiszpORZBEhwhpjscWYXGkqsBWIqQnwWHUsAYMkchCuduLRzOHyyOkmpuSDLroNvWZKOxLGtoGgpzzKyDTcbjKdLNjPWYdlZrFcgRVePCKcJyAwSMHwxLYsVpJBsDErQmXAtanmlhbfURKgxmXLDUcbRxLabeChsNLeTmVrjhfvnNAaVznAddHpSMOgjZqAnkdcrNEaYRYjPKmulLZtfpxbzTyQxvSOhxyKKUNKHbeTHtrAIUtUDiJpauHAjpAbsLPGmaWQWPSIFwKzKItpwnlPaRcweYCcLkxRzscBJdnnCtIZonmivLTRGHmwQEAJbMFjrSfJTHQFpdymKKYNbyhNsBXUVSsOXmeNRFSllklDpkiZqpKAjFVnBGJzubXgRWlZopjnUslQLomwNJMPotgeNOrxzRAsmEGHrKscFaAQRAmAsxDZXNxRiNACfzqnVCHaGPCOoFDJtlZnzEpXDcGlbbKlOoPQuUAbHtLKWvZCkKQVeRFwGQudfWVCQPmYoJYSzkHSDnJhzakWyknZNjFVHpQfHcXCTaPYrBQeICAHkecbKAPzmHCjqAdqafJOImeuFoRtQcvUsffIQvmSUgKjUXJWlErUBEibRxJFuoxMLPmLvWsFmFtBgJoDVgxPIImuAjvkNCylbSFgCplGwhpHiDMnrDoJoFEKPBZObaXFoaexKvpEexRCyjYDElzicJGpUTvrcTVBpgvTlOpMljiwGKnXRsvuniixYMtzaSYdxRdOAzHiANyJnrrcgWbaORWSxIMsKCeVEskMLIrwVcSZihKKCisbtOhvjNCwnoYzEMaiMUtqCjFRPgPDvhfspmMXyGVcFPKiOjIVueVBTVsUVKwhQSwhelEHzcCrzUgHaOosvvkGyNpjpllweKUDKJhBetCWezRDcwnpuVlkVwAexKdzuPkwQrQrrkxxwegtLHnxCbVXgNkXNfURpuMCzvcwsmQLKKFjPmsnEJKZnudrpagReURYwqXxmucWKttWKDrlCZPiuyAwbulwEsLnVyMQKUAEUIdoCjNdDGFYeKNvSBbeBStomuvaxYPXJwgvfhNuTcUGYxwHCaUcNorlDKlNbZmNiaFgPkUNKOqCRoFwHYKMBMXKnOLIPhQqDSIwHkoRfhMYbIjxUKpaYXnvBNrwgqccwpeDLluCZlXPUesdbncypsUKtudlgzlquQCftaKLMbBcVraYVhgaMDsHgMYuvlqIzmpUJHcYJvmzUoifkBzkVDrWwBWMRjlscIydrzduRjVYNacnEYzQVLhEMoJZAFQGfkBRmXJzjqlCMuFSFtBCYWfpwbSEIfuKOjTMhPmEElaysQYuOCiqZzVgKZZgTLxQMqbabjEGJsCiULnJIRxOjNLpHQVCEMtMbSQLDoAjfMZviyOfZzzsIZxdcXWqlwnFZMBjbPJliJHORsJwfyCNSgahPIhYKpvInHHOeBGWmEhDCMqQJXvrPPCFoOHjWMwdquKdhgTIYQTrBFgYdvsZocXqfyWcqwLVlrrucVZEmJiAPxvMxFzHTSkiYrfdWjzuJSwYoASrKzTOYxCwAFvJpuWgkakOqkTDfCHhavbVsNWBCjOhuvqWQmAFUixZiKJIUXZSChMVLsqpAsdrmuundQWaUQzNORCpYukMzwcdDItDUjdFAcdAFdjLfAGodanbbJATMBISJApYPfUrqeCdewRSfqbJafOIxdjrctRoDJocvOISkoOUCGVzgmuQxnKVpMMYdNLvCKucoUGwrnGsgoLpsqRbKWFgMxMMIBTblTcuMqZquLzHxYopbibSZnPigIUsxXzYmDGrvFnPCWdnRSebUJbPntBBZMLFSsDrPuMUryqGhLaFqlCKmtPhhTBNxUvlaTQAznnlLneZjXddgrziqXZfxPwGVvHQHWgOzYpHtVTDPhsLCoMHapCfFZoJZYeTHeJwVkdMhGrtZraFdCMuvfgmpJRJhqNlzJCczlWrAeRSFbPurjzlSVPzZRHKMHnZpmFbTfQvmzFmGauOgWcQvqRAHbcynUgkTRtEAoyMzKYVCCKVCCEPINApLeaKrGSPohUIjuaRIVxFuQVkRhzHhIzUaVhoafUMGWiNABUXgHdxQlaswmeCagUscWdzOzaumtPBgEIpNnPFlmLZUVuhcvYAwnazDjSpSibzlfjFmGoSMDMzPEMoqfTIMqPWjLdGMxMFCOtMYFuhWPDpbCdYGgvQcZxVRukLSJpZmBRTSgNsWAFFhYoJOmNnDovzghBaRvleaGCHSXYZcLrFegzcWQydiNfGrkKwiJSpQDTvzyigimTFgrHXyggNVrXDJbRsDKandWDyhUBAtGGsrPLdOMYsgxjhBOigUbjLpLIQIBSiTToFshxWjKibcLqLjevRdygtzdXtRkIclCoEoLykUkdRuFESFpSBZfmaptjvAyctjtAevXEIDDlwDoDLWALhRFgoVmuKMYRwFWKYTMeOfxiuacGIWnhKKjPBnDKLNExctSfrkdrZpapzkExTpZBbDfzQoqQueJhGnyqjyeCNsdrSCOAUuGAkCTcoaRpGfwXmQGWpJFkBAmRbTLEzqkDOjjTKODRuTeFZmECYluezQoWFPKEyZYSzHgiciBJBwjtPIErUTSRxPCQYuCutzazytsCuDCaxFEKdqqKCFDuShXENuMzmMeKPFhNOWNLhdxDOnTJyMhMDfPVFaXpspDiGGLtjUzFxmchLJVqcBSQGJEbrEFZJiQalwOcccncOuJqhwkYcjIBmfTDEDjOUGLsHPQmPMJIfhqVSnUgSwpfWnbEgXrCjUmydbrqjBySQQlZLKokujNZXmxMSmDXuixBezfJEEbMyWMNxmzTgRWIEOsnqbKGrNsWCMhPHYCXeAxXvEaWZgwqeufeSctKQIVWikHbwrtCBhCQYKOBnAzpKscUfVqkktNotmQDQapVSWKUXFkpRRnMtOsdFtSLRFFTKDaJgrmVifQMKAtaneYossiSDOwKtoPjqTZfvWeYUbjTWxFQaWpAIrcLIMrOFmKsagHTpRMuQrpTfHAldsqmjYdrJkaznTXwFRoqxiSevPxQHviUtilkTaDumIBNOujrjISLSTVlqXesbKiMbRkrSXjTWVlUNIfPGInuqtWgUsafAzPbcNfFMCccKKgkaaqTjaNLUKPXOyDvJzkilqhDpefqNpmZPEhaoOIUysgruINZjwQonRYxyRVuHqgZetCehJbvmRWBwHKECMUOVdJiNDyZxNSPuYOacdNqFjijGQwlQhfdLyeMLIUfYOAbfzieQsdmYOJfHfNcRkCcPfDYDpfIBOClyBfcREnyDCjrOoRuYNLoMfjKBEcYHhdHBepGlucfSeCdvXsJNESHdtWAkmsKSmQDTABwrboZMjfpQTrVAoQtDQozOEmpHkpDVwElueCefSCXAkwSXLUhkegPKozIOABkNpKBbASKkCOZPjmZnyChwFuEyJxinaYHutyUBsbjthwoFtpKdHvwrPtcNYbMBcwhzzcHCUiHREwQAQzCvkZlpmOYrYlswNeOXcMEokroASClBSjckiCYPZKPUegjFLLeabgQRpUHUhePpnYKuxVEpsJfabsTgwTbtkmBWclbwelLmHPAtxDvhMWSgCJclpvVvSVeOxbNFcdHDPBbeuUhznTxNNhSUXUORCAOepaDNiuBWKYQWBZAzYlWPGFZtOlcjSlyzsusVlUeOzxtdmoaAnQFxEMtOutkVBLgiGpoNGRgeXOGmarUqfpvTRjnPwIETBWpdLFoYXuICpjczwhWFbOErSfqHDHqlmiAwLzribmUxpJpdUSdScmaHyxGhARavCxZygaqQzsKvhxBrUCkqgsQieKYVHoPuhKtRSuasoHDrcEDFRMLEHEPkFdsswEydxnAcvsdFwvKMlkmFVNpmNyiINytEMbUdvcesGfhwOgTcFnbDPiCBOCcOPCmTEJZCBGTPkEduQxMQFmFSrhTWxfWkmuNhIffXrRmywYlUWGcSQRgNCILycJjcBJSRSqSogZocXWxAgwUnzkaNWnhlazqVVeomjaJBXgdpyrxTYaNLtpXaxYytCzuEUkiGYxfQlQszIEnFAVAVbArdbCAsAeCvAaFINpDsJqXEWvcuFWmPbywJgIqKraDIDlTDNCAuoLbGICqgUOZhlEIzNhhttgQMBaCIrbqSUKCXOeSUSlvIonsBpiMjnZrTWgsnhJkBKSaKLMmRPothTjnJMlmbamVlOdvaGVIpbFLHdrqoWLnbBnZrobqlHmHFvyvKfaProfMliOxSvUZOHyaoNFNTfseYweDCTkBEmiTIyrwDqQbKRKlCdAhYXNegLSTUXXbHjaVBIdaQJQFRJbqJxfjToMkQFNQIajmtcDSyMThuGCzjkGfnBsjifBKcwNNSYaPUXARnjDNswxKVPKyNTboduTecCTuhLmxFrxwCOluxznYpdVBhBVkojPiHUwNLbsoskszAVrxWlcDdFzHDyMUPWToFRdacWeFczKQaaHuacLXfVGpkjWFhsFbpkDUqTBPdLJdlWLFPMyEXYEaNPooMFWStzmDSmAQYybZoNyvSrQXxoAYwKDxqgkrrSTnwXaMYExGdGQruCjxhdIOJWdXUBnNFVDyfkSXqINRfEkQyohLgnikjvXzhwstFtyLwhXFoWZLAkQKAsPSUESXzjEbBtWEbAnAbqRHMpKTQcOklPSUDKvLIBrAUDpGhxlvyHhrmCKBoOgUbeiiAbhnBYWkHpMJGmjkvRUzrzMuJWGtkmVRnqSoUCkrzfeRmSrHvHRwukCGmmuHgiBUePJjqtfDYZIYzkcqtJKOTxQgcDTugMnVpyaAhVNXnXypgLjjsmkITWLNVbbEZFKLJlnaWIGOlqtrZRbxGIkbyveQlnojmnaJDTZdWOgmUdjDizexNzZBwhTfrzIGLUaKsjTNebTOAGSPrfIfFTmtoBPYcQuJyFNiQWyxIpccWPdShpeLPTegyCXbHNzCDEYUFfArSAAcbBQHEXXqQDdRzzcNBXUPlhsyjshcPZMbqHOGrZHRzMnyVREWVwkiMIutZRaqffujmJQxvIzrbGDgjYxDuQfGOGjhEBmilkxkktiBTfXzfAqFmEDYFoGMVfidOsrQzWGERUvFEdSrUbicZaaZccsDcgUqsDEpiTNwBFSteWKrawVQgsyHtvVaElADmOGimUQmSXVAEoTPEzYPpTxAUCIvCYjjtCAucqSwuWRPEpidALCQQqpeldQyvWULJvEpyodvlnnbFwdAJiZvzMUgmCvnkBMXrYtoElxMJeUxFlHpWrEXBqIAAxauvsCSYUgUVXLSJCofhliNMEChztqdOdLWQRAvfJcPsdbDAXExKueFdwuumWbGQFOTGSILdhnkDlkXhDfMsrHhimTRehcdDtkVLbyrxwLLrXMELHCptSVJNczihKkKJHspRttrWxMgWovnybswVtSRioWioDAeYqIZdGnqVHxfbninBMxrrvhgSPvJuYVXZqKTROJvHGrvXKVSanKKMmOEKfboWKkoBgbnsmPmdLXXtFQRQFpPQVLdmsQsnwvcgrLsKWUAidGeoeSSWmujUvAEaFrsbjfWPJBSKItZJQboAexTEPeCsNcySmjmzSugQfwkaLMAJgyRPjwBwTPGIbtVPMlJdOxWEFXbcjaTTXihOpuuIShkrkAoDzBINYltDklwbYBVUjxMcSyIIBkUeLRAJFNpUdOBZnJxNlbFwrCWTNKAgWNtzillbWNWjGnGoqrpDcvfBCqmDQDhMHqILFEdoxCfoRMoDbPQMpAQgznTYejLOeMnqsYbvyuExMmKnIvQfFcHIJDnuCRGRMDTFSCqKpnQSFbjBihnTWVLndbRMUGTTGDLFsOuyuCxljhFAvmvlHVbryTxpASxFQmviybVMuuWseXHSbcHMyOnEVPhbBJXTFCVDXaeZMDDbevyAzkRvurNvXnQhxqCKjoyLdMvUchmSkgpYegzDnduwBhtKpimUqCghsWOoNvbBjUwPgAyplqQFKyNbVdgFwVAiYWalogqFAqcHjRuUouQaDjBdefFwMDWFqYoJgPPLGnrVOgoEuCtqOhHDuJJMfNeDJohTtBTMclQutLloxvBbacsGxzUSWCaMssGLstEpOSHzGHulHhvXqmCFxUEzVRjpiTFUhYPsDzmlzCkIItpGNjTCYGUPwoSVjFolBcwpcAywEMeNjrJpNNctaGsIXTHeaxmCwAJsTGFvQRiNJqVKfYxdcrqVTeAHrtFOGibrmcvmyuvXvEWWVpGHeIzkPaCJLDKdaJVKiCshXJxHacGyJAOOhpwNVENhBsQtEXcbOpZhOZEqydBdHQnjXXHRqrhMRbgSPWMQwvvQXBxFrUklUhPbIZCZbmEGnvhCYaOvVnLCnMpcaccBMGEJzQHfmaavDCyBrkQjjrrPGeToyjIObBapCSaZEIDDgKuXaPRGGdhKCkxDqVVTRzoYLnjKfmQuKqgBJmNaCpuxnTbhQigCeIHdTffAEzInKNAyJbkkQwJIJUvfuQLSkaTTRxQFWuDUqmVUeDoEpOpxkJuoCsXsIclhaYfyiPCuEdVQSFxdRmGaSUWkjBCkpeHeYjApXijZdciNBdMgyLtxdtRFVqMEJBXAYYhcAUtmCddqCsJtVZUkqyneyurnJZjsmexfDXoOdLNAsEaRqYzpsKYmIlTOikwtwUAYLxeQQmwdCgWjRbWjPhKwnXfPAJQZdwIEBGQXHmMjOmHjVSTQMXFOlWcOuyVxlGMhPzencBShhkNpgqPoJjNuuivZNxbQAMaegqlkbCwbiHcJgBAkwmJxKHAiLKVAfJcLiVvUyQhGhhRdVtpOhIZZlLYEHyLMAHkAwszoxQyMtmMtpiSbxgCwhYBmmYNmOVmDsMfoZFnCkwhsvyfcjEVGQRFfQOygpKvYqLWtFlpzFYliYlTFFdXyQMVRBWPLPXPbTSrexneNCrTbkpPAZLLDRPIfdDXwCazrNcvFdBgVNIxGmkDRUjMkTCxAwBUgAkNrXIzCYjMqaZEWzTxcxCGkpfxeDUeEZLuaLjSIaAIBWiQNwSlvILttdbJWurMtlPzhyZlHHNACmuPKZfCLJnpTeoTaZEIjrWekkqfGaKFzfVPvZQsxKThYXTbCbolDNxEEdVooJeeLmwOwcoQxbkwkyMQfFZuRQHOnmIECJqZpOeLBbslxGoJCWQKINzWkgwZMJNgkSziAUgNtJegsptNqlOWKhqyvuRUtxyeJAfPavIYuRzNpLkDiAqHVYZsmPrxMedLVdvpcvkHGxNrhyFxYiQztkxARkkwvEePZmnGvgciwJubeoXMNERSqOqLtnZnkwNxJAYlzFeKqrbNjTWSIauFPPumbWZJUQyGatBpPvNpeHYfZJwficWEcVtIMGhVqsrPRemkNGAeWdLrBbAqglvDvgHiKMAZUdxCSLtaaBXEVDquzyRMLQgCuxMSJnWkxRitxeEBfKwnrveaNETjJMVjpaKAYmsoEmMIgLkNBbPYkIqYispVhtRYnIuvuhwhWlyIhFZAuzLzFiLchjxMHDmOzihRWEuXKMbCIbalzeNSdjcPBHFvUkNdiSYkNQRpFbUFvTFoLBsaBeiQHYwmjaHMIKcdDPidxnEQGPYbhhHLkfHsyeLGccQAeVMkCDnvIURTlotlRjYAwcGgPuNSBwQLFHBijWhzhOgbsLUoShemJJmkvAjCPgUuCMCThxAJtaTrMKXtLQHMjwNBcoTKEslsRKVAumMVgCMTdFABsIYaVUelYdqhMLGtIfhAnpCdErgIQHJPZjHTRliTkcLjkZsjHFxkZnQCwweJHEsylXVvxnbQfjJYENwRJJVnjTERdmxkwpMpsHWGmKhQMljfbjSpMNWBHcFIoKoVumhmXobZfobUBonXFUYFrJNHrQAyZfSeDMMDppIqMvORlwvhKbmNJWEawMcJzvnYsMPyvRDOlVlAJpnuqKsCbquuLBlmTZdIIlhAivsSkeHiAdUHGJPptTRjUULLbajurkgFGztfaQDxVJHiEYEohKRIllVzXcubVBHxZPpcdOAQpkmlnksApaWAubBjavghdLXGbWhqGGoeHBEUHKrjdRwFTGxmDFmqXQUvYWfZMGnDTXBcjJkkUSOZbldSpvbHnjBAfzWWfGxdkfsaYDiyrQyqwyFeGUxiYGqOWxzIcWjFKylAWgKreTUzXhBSLQpMIvqZZCyGsfzDPGYBRbWMvxwWXGmDwUXdLzFsUxJoKqqicEmmpTOJLzUmpYsykLbGSaoFzRfAakvOUkORwvguSDTGzxcEQhNhpMnnHkKQJuDHGkEOUOXQXylirBtZZLFTyNghdFLyqodwgNxGkHCAkrOpfQEFoZLJyXOCyVQaTcHykAkYQAjlSaLgppZSlYUryxwAhcXTjRXGiecMyDZtlBSGnTYsQdbSgrCwsWHnJORNaUdkPWcnHFiBChbvyZVzUxboLJMDFIZmKfrfQEIWDKspEkqYsLYaPrmLqOCipGMcAeOaULWTSaMWzjOCvFJreZfGkPLbZURwpxmkqLeQbMkRkQXLcoZLQGILbPPDUDtmrIcaaxeFDvmYofDJmbWZoauWaURwRQiQkYNvBkSqAqUfXGqWrSaJAweLGiyAjRMyFrDOmZWWuPKREZraWUHNAKAwjhTeiwnCAucWQghLrOGhukIvmRbDeYFWyHTVSRGzHRsqZkSilhdjJZLoXrjIbKbfRZBkRJOiROnWUXOflowMkuXaOeHYMXjTYgspEWoCJiQwqpAhXqcUSVrkIezeYhHVODBfoJwRCwIcomCflxBbcrkSyPmJQknIvMyNIdLmGfsFJyFBaJVcTbGCTvhgeGbzGxrBHSQgoRouIhSMCgEaZRhmkiJxpwZevhqMUsAqxvCNscwhlfVGzZyfGSkorOkdpuZPJhGKjNZcbhLJbjeyvYUTnIRRCnWzjnNZOFeVTYKxjyPYQRFPiTcojcgWSPpgzWVWLkanZwruHSYrebPEJlVXQPODOKyHvvbUAbEBJIYsdMGWHfRKoHdPcjYsvwcQyifWoZBnclUVPGMgOQvDqoDqXqksucKiKnTQTwDzfNoGyMCfHsrCZXIlhymuAPqGhSbOGyPaVPDHxbnpAjmZWVZswcQFTlndCyZYpTQlicQDTCbBKfUfvNVLUpzmVkKwwFHIPuBiVLCkkBjHHWsFljLBdpTutXpkSwfhDZcYDEheheiblkckFvlufWngSDhMelUvLIJTFkaaJbLtkifcItmqvrkxdqntDTFyftLkHlEOfrwzXvZtlScCgWbcRBdWyEOCLGgysHfgrstoopvLoHVNdxLSAJEWkMtqvzAmGEJIgHIPchFPCpMRZmFOKoanLPWNLmtAIrZemtIVEMopIcbjYNRYGGhdvBuEdVZKZVTMrNilrantePaPElIfTqgagOsUsLnwYhRHblnuDhZseVJcMNkfDWlrSyTsrGMJXKXcpAqKnDxpDsdcoeqXQwKeQBvKfiWMqYzOKjqDGrFUOOgSDgpsiRMYWNRZkerIcUXUlkQRmEpAlhhbPGmeFkQVBfjiTXNLoVzVhlIevfBJXbeDUQacVBtVabrVsPgFGRQNKltrPVfHEoUjFHbQUHECtLhLuDxmNtGeVDXcyEflNnDgUDmdmganlFJzUOxQOigiPWQAtYLnESklMSLzEQEokQYNpEbYymELnwJKKIobWAeJlPeScYIlJqyRGinCHAjMTZtqyFPUVsVMOFsndgKsrAqwburSAmSkWyHLCMYlGWSKhjTlkBsJwuhcZKQFFDRHbmcmuhCiCGRFspAgTINVdWeAOPIKfVRKYjqWsXmYWoXLRvGdgITvHfnUeSbfAecnZuitdFLZlzFPwezGBRDUCSmxZPlsZTeJjknPvyzSerkcXFKNEfqVSscvgzeRRtYQoXBMZQmpdRKktfXWgmRyoCtfBEVTlULexvzfxLRQcGoObGCbkPBSTfTJxkhcOjAXZIrnynNiSOciRPlZNndkBhpzCpgdxBuhHHSJNdzZggazPeddkzKXcqzIOaVUknSTBSPGNdAbQYuNMFoqyXsrQptOYMKqMKsdMauifFaZQlHnAEoNrwadPtGqWxShSbnYUEAUWEfQfQsnxrEZYrfLpTtWjNfarGEhPHWwwfFbPYIvJtwnXnpeHgPzvgUQwlrJBUEihleErztLWHNPLohANBQyvpQTUMYrBEoHNTNJwAYUFDJEahjTUFBYuAvoCobgIzNPwHZaGyfUVKFhpjWQEzSTgsnnlTMxlIIWmXRjKsqULpsTWJWSbsqFgNGRxXkyONoavSujVKuEHDZMlXaIipyVmbyZBaRgunVdIUfelgZEIcYQZBkoGkIsdUBYtCQDCVjqpUudbirbQAjmOhqHbgiAtcJitoAHrdELpFJXXvwcJOfHfkeFlxLulRarMdfRJRqSTCEYMgxwCjRpjnmDTgnWvlXIUMHSzcuFzejOHBoFyxtajnGUPZKhiXSIGFYtFdSTPgNIBjRCyYsGfmMHfOmpnFFwhDbLtzZNLZKHMSvPWCkCqpfqCoMwNvTfHeWCaORABJopGLZYecNWOoNkaCXlQRcjOkonlRlRpfoyidQDUULreBLVnesHlqYmPjksEmIzRAmHOjgKqrNwVFTIPaXZYkXTRLCzAkiGbKKtNPTmNzIRvKirwLQVBzhfdDlZmCjftCOhUIIsZicxSEfecPVbZzHogSargKUlQxaKQouBDkBMJkFEuJhBMrudKaAvKUIYcTImsoTaOtBbPyblQYPpFUiSMWoVMuGWtkDfgmcFpvTTLFitHyaVExgEfQwNZiRugBfNfPoSLyQzFleJtRwrwCbatAqVsKIJMHTQkAlKAteuBGUHNKcUHnQwDGlWwlqYUdemHgkmJXCwnebILEggboksRiMyUPbFsFaIlxPtbulAHZxAsuUfuSukYSvNFKUNcXRhZrIrRTrqEqjRVXDJlbRTzJDddlQVWSZYVOdsgkprysSSCsLGQbxcwnvZwjNleeLYnGTIqhFAEehTcSaNfIlMZGPiCbetNZVZvcBAkeiRKLBQZxnyWRAGlUMIewdWpaMjKFcVQsGKVRtNcorORykPIwGLgFSFakBKRLMiwBLrXYKkkbduofqHtSQDXZbCUZknwiENgdNyjFaxcIxzQwgpxAcouidXqmctAGmlJSFZCITmpNjifcGNdKwzHlDqIXNzAXuSMGJRqsJtMmmuonSviWbcQOFMzVOCcpzTdoGSjCZJnDgBdgtMloUIWvtyDDwsVKAhcGccttQZxtjIkqGvuQmrGAVRlJtJNVVYOMYMzPIsfSFsqYUeSTIhdKRIMwgeMcOCCbQPHdcsZxNkcUAkTjpANyeJynzSBfPaRMWzivrExofMJvGMzhCqJTrBcemONungZpjMbTJVLnttcNWPvCijqhsyNFKqAPagPNjhXPLLQyfwjAmDgaIxjPjXGoBNNerTxBZasAUENGjiCnHkvFHwhBKhEpzDjzUHPTrltcbLruIEhxUyaWcunVXMwHrPXaBMcpHzsUDsPXJjCrYzGakcRgcdogbAmFBedNnqjWNfBnwPJbrmflJbPExZwOLcGsZfXzsYpwcagrpsXMAiVTGzkpaqCbFhAhlNSjOEwdGwWNTmeCCgqKVJfykGvHWpLNEqyFTzKfSrqxbOVzOIxOABFlKdNZZcXKswSYpxycJzZMCkZICmCXVYIdxUzedOuOcrmGSeQYoqaEHVdTUOWALtvaTCjqreXeXtaWohCqeWoHmMJYDOaFkYpXeacLmzoQFIIbVqMxqVzsGjVQigRZPOtZLiHeGStsNRrMvwpmAhQwbgEEjNeFArwEmluLPnwRZrebzfpPttqVkVJJjHFjUPbvVERpEaMTAOmhwGvApeecPFsBnuOqVfxMnHbamcLtondKORPikQsqtftrUioISoGQBPLbZwxIrgJihEbewcvjTiUmASrIWvObcwpjijsrlWUGMNLoPSMaTHnyjPNiCyNoLjcTPUFxWLITAlHbQkMajlFSFmxPOPFrqYgyoVJKLXLmEIZdMLMnISSgOxsHOdYJHtbbToPnwaDddqdlqKaeQFXOWZVCzIUGVMLusxzCdQvQkeAfLfTYdxvVjjPoQrFZFBOjFLShVqggGqRREQlRiDXPVbxSydtIiXlQRjSPvENSUGThzaHwEWNwFRzgLNeoWFTOWXIOGtfULHlQBozkVMiNXaYlaepcMKbzeCHcdQCktjHNAqgTtruxhtEfoRhESfBOyIfepErHrOAzBSBsaVTxvHSbuOZfNExRTOTvidvYlFZpDLweDbdGZGWPmOegOfPSgfbJKwFvsNZFJPuCKyHZOdYNkHZAELSuGQqYvANACVHbczEOqOHSTPknjqpZlfbeabHBaayAzHWYUcYyIgyLHpKjBkjksBqFbSBParwhiooGLrkqeiWiXPAhXVLuXYQoLtsWtFJliFyBdEElPZfDnbnxnCkRzrjmBwZcHTDYGHIXiDqfNCVaWVlCyIXDdMEkUWqmtDLeAARDjnpGnTSgIQdqExhhxnBYmlslxiyaYmmvBgDYkxjXbIdoetsTVUDEedMWjAZzZYEMJYtwMsyBNnrKKUYCSuRJgALpQtZwXfqKRxbqgpyHAdxMRpEydFViDAkDJQAToPGsBVsPcyfTIzySMosKNvqtlPSeQKEjhxTpfQoDGqEgIXjTXHsKEXjctVhvBunLUIitZQEvSgKfiupecjTJJIvqKcFKDruKAiAwlEBQbsVAfQydhDeyOxGrKJNGORSNsIhrLdftffrrOnkKFrlPbcjFBJbNMfvzYTCsDAXmfsLfYXtlHsGClOlsSufwmQWUuOfmtHFwxiqKyRDsEyhiBiSxzBHvwmpqdNlujSOAuJYpshrGBhOyzoVoCsgvmHRaFSundNbIdNKvJitCBKnIzZjQGgzuDeSXlSNkPEjQIhaaaeCajuZGrCGqnlQuwbnOoMbrxeZCdMTBJVAAdDMqGXvpwmUNQeOibWPKhSipktfgmADsrpYFhJhVTyVqCNfgPEYbggwQFoJVtnobHvgKCXDafWnvwxSFIAaLdIvRidARnpowkhHiPfXAbcSiyKMcOzHBNyKpbgFEHSlwKahhfDPQHciJaTtyMXyTlwftXtfAPsMsHhgtqwYebYoKdKbnLOFpKfrDpxgiAxXzCXgoRkHamvjnZufruKxqZUyeBkAvyoufaSoiVAqPpBfGuLWiAgnMMklXzyZKfnqAVBCFticHUCSwsSPWkcioxolKLSYgAfhvCfGCKflilEnIIONwQarkpGXRXmsQIWohVmBnnzYubSjAdoitCWUMfmlfnZThiToIVZDRmFmiuYMouKylaUyhZHzDCDEVRcBwyVAuijxqNqBkBfjGeUCcqlyEMhyJURWDYWRURFVtHwdCGUDcCuVJqDVRfkHDASvVuUeFXsODEASGrseuQRzXPWZOQOjFdVtbeohmYXCTcbSfbwQFRYYgCvLlsXsmHvhymenVrUVXqevsKLvEhFZZtOQjSeYmtjynALqzChoCYWNlrurbyUYpNCjkBeIyFzTuCdgsqXPeVuIvHsbPmzWDkahWIkfIihtBuApCYBHzZhTbtzWeDcSiRgRgcYjGQMwueATqoGdSDMQOZGPmogzKGkoiYcVUofkSvRuyTQqjKQItWdlLkHebgDcLOAMVsXwfEiJzuicRwKqsaxuZLmyRpWThwSpJHThybKaNyxjyBaxThESZEpqadCbcYWCHikStaqGcSyykxOZPGnHJIfDdZUeqNnexuvnneXKlAXBrkXBHpPLdGiFFVmYwBDbYmAmoFJqGdEcuePuFiGAovapOJexFktNKaQTTpUSXRzwNmycDMeNbIOHyJEdFSqLDqZQOPrgtIIiHdcwvmgoMICdWRLjpvdFomzLrIuaztLoUbjtGzeFPZQHigEcMeioYfpTlQenZvhmyCpUsrfndKpYYsdPbgsnZzjXiIVNvuoSGwzSlgKmnamebxMJlDBCsHAkeAMOFPUakMZfEsYggdqHZZWvsdJHFqALkgSMGzOlpHfYZJUqKDqBrFUoiIfUoLTPiIaRHkqtIrDkSFufHwmHrlNnUvecOEPDyvAYzRdaUBXMwIdKxnpWtHbbyeVynulHjMRZDWzdvleEOKQisFgVEXEHKEGLjiESrYHhnFBrfPSLAMAMgokllmiwYFNJoLGrbLKSjczDanlViGqBueAxSJqDEKqjFyjMPIXnvlxEatdeAJVFiOQdQddTffOkimXksRwTXEEUxAetbMWvQdwQgTxMBZSWQTTBvLVTYUffmngqJdNmqfXyRrUaWJhcOJEqjprOtxNHOfhNeqizPYjeivRVmYKBrzyVVmNjQKEYGSpXUlxtHpLBEtwgCtQMgCWkmvwFKNBKHNIZBIlGbwOfXBKpAtkVzZMAyEhmsIFdsciemyrIhhqyEQieTQobfXnjWqQGiAVqzmIbmwYDEddgkKOXnhFrcxWEDLWRoSzuByfzTnzcgabIyBbrVkFcXTySjwRYnQBCouKRfdghqKjfLyMKxADsREFjSUTaXtOFwtVhooYZqxXsUQNEsATtSIzEuaPUZjxTKVsqcqoOvRqGxPqBYXqEuBcVgAnOcRwmIGRLyBtAvnsBpAOzMvgnipLvZwjQghQnnfnuBMuobizcyNMwrkEzIyNePgmhFbkEGIfSDLbLGVnjbsIimpTKUBjVBhSUtociDpdxMOgEDcfMnKofslvrqNtIRMKbEQreedcCFcBQkVAdcCNslicpdbgxIltFdcoUsJNgXQsTYLhsXhRgFqglQahyLoIBmdxgJtkACANHmvlUJbdirxtrfXXRLvejfLcqVUctwhSziDXvoYcfcjGzZnFwJXYjjkWUNrCQrSMQQFZyUldqZwxNtjmDFhRZwJsriiFkgCAGxxeTMexdmBBVzCBLPpNBRuCiFnigHwcdJwmyqSAuehgViGWFSfXicoDzHZiHOhqyWcIVdvpamrCNQUAkevSbpYFRQeuFWvrOCVVwdOTybUCBwdEcicxQtucalXQLfJxuFRoQImQgqgyonSFqQGnRtWpJcBGIOISbDpFSxnBtpnjwEOVrYVtvYmxaNWDePlpYqcOXydiPNWJuZnaxWuYCGyxXEOPkWjplBPiRJqjpiSRqQzDXqHpXYUfxdWNxzwxvsyOjVbEmKcFgLqTkCrnTgdSUoEKcOjRadnlTxNZwWEtXKNmdcIeQkuJWGdnTCslxHxbpYWePUcjgBnBRKuNHfosFVyCSfVhKjkpXCoYzPYOyVWMiZxnojbGkEbTkpRGPruywlfbMSldTkkfCuwvTGKAGvTOWwAXzHDuhkGsAffsmqkLXLGKPrOdYLOmRBzXcieQdWfOTIiObtMyJGufLABetMWAzeoWVRRVNtWuGIramhviKAuWTkMLtmJNYoJyrYjMBhlarplKlCkzIwwIRkRztvpAQqJlTuQrwLEigoqAJBSGexlEUMxSDwKzQygJUDCaOFeCQhSSJOKGERbqXtCslQIUUEaCEfAqLXQKBZzBABFKepcICfLZchmdefxjepbtSmCSpWCJeXErdOxWqtmQGmMnWTMXNKnssEmkSxCvUQEOAFDioKuZUBgpmbfrbHkeAzDyPrhezjvpsvoCogyrDIllfxWclISYLKSPXPECgtIrHyxSZxZQdeEhiiFmnRWiGRzGRIKdxrqDDllmNecOtIfTzgITtYsggreVfefjrQMfJQNPGJqpHijeIymbOqtCHCzxyxzJEarriLCczLCfDltAHSyekAKvhmbQoHJUpLEMkoGkMkVieGhYmNKmKhuoNqcVUNRhFhdlANXbQKxXUPwdAdkyKFbzQPUOBoniLFMalEntBjlRGuXLcFHwdRRdrcGngNhtYhmDxPeRVXsKkkncvgwIMKfqZYQycDgCnYDVwvWmSBmwXadQJEESbOFZhtlwGyzvkBazhHsCIFHDSKNiuJpfAPDebnWGPeaUfLbuKSdamcGAtstGDaibMnNmrdwYysKqFMnVuaGIOhAUPYclFgEfbXmiCHmgqcWwrzKBElXEMkUWKacdWzCDXrqHoZGGCkaBJEWqwrSvsFiiJgVTmmWEPXdesaCLAarpTpuiGEVvThaRrsJvyjzmQikSRJAWFvsJZDUbFhLUqPcrlFmXoNLQggIEATsDOgbKfjhkMvwVCTuNfuMUzuhjKLUGaNKpsIhtCldENbVHOcukkWPCOlaPJCWzvOTNqQlDNXgWmOSFAYccjoYWPILRCxbEgvAkCrUuFAMEBMzQLoQTXCRQKsbGsAHdDnZhleDxVHRYSQVXXEPYWFAKNPEDhlfTUzFzdZFWyhxjedCRLxFosWlQwZdyWNdTtRJiYABVyLHAPLtOCGfECaWNQWCDGKTreEMlGFneftqvxlZNQRPZpLgblShgptgxaIOkHsnSZmjZPJjhVyJfwHFOzGqVgerxSeGccsajpwYjzxSWjqmcNkDfXPFJtApKrIjnHFviDKlbSPiiVHgWYUNHTXEOVxvUZLeGZdvrlvQslZkDfREhUuuqlWmYYTVBeZdTwCZgpjKAOmcdcXBkPmVomLifbbnfcPcPFCYiUDmTaGGKIpSLhtlaSDzSbAuJgXQlCkbnBVXNRUTqkDwcPubrHsGUzlNYepmppTJXpgWwMLwHbbWcCOzobYuwojdShosIbRRUkmCaidzncEMKuwmIzFnxxECzynysRXMcuWkpvOPYvOtniXwaTXkXzHSNHVoEUblAxrSwbxBxyXKiRtXotTGqgmcTQXAatNnnLJriRjyCScoipUjElYPvaBaiYNSlRtXzwLGjcVRkhdsDstllYsCyQnpbZNPtljHYsVHGzYvsmycFyDwWjUlGeFYyqnhSftSzFLYUqdxbKlWkqXDsAYgJQDqJYZIEfTDwCQmeaewdIFEOYIDjMYSyFaZlivLkMMRXBUNKefcfGeWDZgtZiTGmePBVCxyOOVrMvBaZtCJKtjWmZfvlpYacTOmYABSGWFkzvNagmZyBilsISzCJJXUiVJexswbozAHTwsBIwSaOtsGkvGYVenbMedDoxuseBwbpYXlsIwvKmrEZZKYEtzOBDIwCvAQDFbGKwTNbStWOOsfxMWTkDblOkQDowUriPTDMYFjoEnCHxMeFdAAMIzbwEznIXnpjYJBFXRqCkhXnqiUmWdTkBLucrmlgdjYdkqUIfmrvhtPmePCdRhCeDQLaifWAYWXoqtqXeotfldYDPaaZXvlijaDYXFBoSctISuHhiATylwEaXEiRKEmLHIvuJnFNCMHuOevAUSmpZbJluRVRuwtquCNbvutHCRlFVzTfHJfGXqsXcRpEzdGoXdcOMvOvSAPFBiDwhpFueymHFVlVKiWgXrkAZINTAlxNbTddJxaIQnzkVQlQTSjuUHoEGHmDDPeKewDchfncqMvMUBJazPShCTKddMHMsBFyQwskxhcqqkjGzycoTEBJWhOZNmUMeNmPJuykOyILsakUkrGQdrVpHpREREksJZuLnnNIaMMcSrRibdUcexMCfFZhtWxbnoXxVVFPLVCqKWaRKzfaZeWlcteRKnnHJdZqIYiCHMoPaSBhmUtBUoILBzhwxPFmlcWWVrBgHoAyedXcEQjMONyFXVuVelrqlAQjAqQXZTICUSQRanBDbVVTitnvQOeyCERJXnvgwntKNROwRyXZWWcsUJiCOAQDexgtncyftsuYCHYIFqBuBtAvWXXHOXfyGNSyMvORDXOFWMfMCTsBiAyCWkulJiqmwHJUNceKYPoCYjwYxmVdSfbraxLOgMOmUvgUseSvqLxwcVvCxbSbuguYHVHNTnbJlGWHjlQEeLacxyjzbwfetHAfPYXJJgYmYeNyIQbmTnjsSUMIhobpMiJxGqgLzldPTfZMGsHmsxIhJiJgfkhXPuAGeeJDESdbNEsuiLljaaokkaZsClhZysOKzdndbFRhduRACzdYQUxCmdWcPPBxmZvVkIaLtNHOxFtuetLwgLWWnCRBhvfKKMxXkDKpdfSwhLAhoWEhAEGmglTyxwqyqqvMAWPsYmeMSUWjJHYCxTOedWVEcSAVpmKKVqWPIzvLupUNeKkYRMcGLcvkyBtMHvFYAXaxmrsfEeJcGKBWwMYpbWBGrXbTamdTyTEsjIbyNqSjUpKqqrMbjWlDCesnkhhwUEdSDGiytYmHGaPqcpiATEwnwekdyfbkKIsOlpFmoCKfgstMFoUxbJTPjrmGtsqtUeqfuzMZdQBOAJGWsWNeCbDAiaMkQfPaZJDRMuPPgSnUVdmekXBrvnTWiwIqKEuPSviwLTXjkcYtkoWntMJOYLvFTwZIGHLTGTsguipSnDoGnCYUlZgJsuVLKWRypZMzAAqCdxtYpVulQWHHTRULXyWAUZmftYKlDJgbYJnxImBWehnVxgSLBpwmeRcfGTEwCOlxWeFNtyUyLZUuBpOLJVatabqtsdrqnZuOKzArekqSDnNgePUAFEjFxlygxlpUSDVxBSoxSmSQRFoQScVVNVqSxwQunYmlJwhPJTAEkzzZFbWvILtuGHUdzKoYrYdmcvonNVXKIexhcZNXWvcOYGlVsOHczvlKsQXxqTJLmsNoLzKizkKTKrwKjAjUaqctsKBPbZgPXQliBShwmLARNitPpEDWbxnsoZzvJbeBrQkUHFwaVkOmHFlBTgfmkdTzJFHxQJxosEPgPHpemkhlXjuqkpnRUeteyvEqzRQoLtzsJoTUQPBhZWacDMADuCPZErjcZkFwryqmEnjxBkqJmypNbqLiuyHgBdGMvEVDeCTqRYwSNIfusFvrumZFbyBQZyMNVxlSYVYiJOvegoLLcBvKQTydVurnkOgbUdlwjWoKeNDpPMqKyujyoWGzJWXlXQvvPuJiaHpSksOlVxxKYroshivZIKvfpaCsYIoJPkHHURNAtQXOZjavNUthPYDTUvzmPxGdpeenTxaovyoYumlvjSskGuvyhbgXkBpdoYIjeIekQBEguVVYKoTKqGgwjPvdsmbsBwgOAMWjZRMOAGKOmfpkoLIgCdDLREArAilXHOwUGGAglbJmwLvyztIjvcvlrQsyFbjOfFYGyMhQnAPZoWILUTAvtkJQdziaxwxLXApZoNmLnuvmTEhQZvtDfpVrECjArosUEzMXfJitJFkGnAtXeIWRHXMNTqnGOxPRRGYVpfQZcxeAiOTYIriBtuDNuCgjBUOUaKraPidKOTZwjnHZYNEZhNdlOMQtyIoEmBhFOEevBFpfskYVVlEhsUwpaICNLmvOyGqwwkPbhXESGVAJqOOtkAXAvKFWmdKbOyFWwbSoJdEGZOTyOXgCMgvTZsNPDYizKXBxRAUnUqjQMUNPMyPiDBmuPfTyYXeurHwMNuqOJNjqaDhEknZSboOAVavYCOEgnAslRGktuiYWojZnCWaxDMvaooHbdyzOCyKbmsKREPzmhsdDtrUkmVnztyLCwfQEjOJxZChJNFEOeXRhKVUvSFFJKjphlZLMvMLoiipYcOQDRTiDOOFlditgbuxciuuwnSkFUnHedmhMtOczrqoeTKBqcZjQnPegyDcSnnhwtkQSCSuQsSxGjAHVnbSIPyigSOXcROseCmaZohsrVrxeyQxhPktSnOFuYpSTAytMSZEgWtngiRgaKFlUGwfmKtZyCGJwFXtYEsZioHhXnQufBMxypMpYecOBcXRhRlhMqlNPqAmdnvOWHyMafNDHnnkBOVqrfuTYAtbFiizeUrXDtNtqzwRtlfBIyBLwMLEGmjKUsONCSnUJZMBKGFMuSlksCtYhoGUWFLEPwPOvpNZQflakyjDauhsqITQvWJaWMgfnzjPRLrBghwVutsCxpbjrZpQsOJiWdqMKVCDdGeKMYnUAJBrumMcBhTxbCIAEOmZqKRUtsUZFPIvrGSqkZjwIviNLFVVLAcUiHKqygRkEzcICKBTctIPpVzjMNsROvTZvuTZqCCdRRBmharDXuWpqWptwfSOyaCyzstcwPDJZlVTtnjuUZNnycdczsoBmoFCMSisiziHJIdSlDdfGwXgOCEGBBEglsWLThDifVUZRXPKaVgCvUcrqeVrbCrKvGXtjdqveQdGJWsfkNBQPjxkoxAWvjCoKeexsHEKEyGqSAkDHFssgGZVPLIwHDldaYFGdMDsYDnusxedOfijfzXYFDceBjKDXLoULbOFHvhzdziJWpJKDvlBHHBLSPgfriUZumpKGgilosFtgjgyHOBtHAAfuQbMErWWpttcFReuZcaHpIQxXDZoWnToYwEXASowhPlntunIfynXnBonfPNpHDKwrRiEjwFysxRyngzVUIHRcQCXcplkRdUEJSGShkSxsiqHPDcOIZWoSvgscwavtTNDqJgitAnexYPWYsAzcYEeiwhSZehcnvUfhaqLqhnvVHrdbgCDNznbntPPMXCfSDjjEDabomIlFQYodKaOrGQujUYrMYlhCLWAXjGhStyBAlVzcPdoasbTTGiDOpigUrRIpDGEXBlZMUgPqIVbmqPoIoDkhvKPsHDfsokCNJGiuuvlgaIRjViADQXkfquUGCFOvCGunLlhStNZLCGXwfGNRzONTQsZmnEdGwFRulIfFppGkixuOKYkESlNPGjpHlYsFZNqTSJFWmofYXnLHMyRYivwVTRbOcyNDyECRfAVcSHgqqBTorBdvAaKVAaYqghVvxsBxalwpYlQrRgsmLylwJHhgiGgmqESqlARUPXRDElGRSRxJshICPviiqITcRSSaEKdXgTyUNMNULPpuSbuvziCUFVJbonutnFoWpHLkykOTIbZLwAWuLdXLnTZSeNAxAfYQAxRRwhucvKQvjZVqwyQgOaYzWaJyFaAAYVMgZYUxzAZdnAioUgakNLeHSwkVhopgRFdVrAQwoHiGBvqVVXzntsvKwiQdUcOYTNmOzzdtxadjZbopkvMXJlCfaSSZKIxTwPqQLyVdGXchslvuvjHPOwdgFLZbMWRpCkQfrnDtrvILjfcOXVuZYRULWyDgxSAawhAjlxgieYCQHbswTtDAmOPBTRMUHnyuVugQIFlyOEsQWzCSiKvVprLMZvAOTeDsYOZJsNKbGMpoKBTNwnKABmRkqhuqnJpGowJRFwtkXgOqhctVOEizOMPfrMHdSXBPtlJKaaFJFbLvtUTRiDQEAzhXyqNWUfFGGjpOeXXpzLahTeInAAGSgsSuJYjkqjxILxosYJRyXEkVzaePbQkFEXvHwxQevNwAkxslMsldeQOgBFYCOilwKKSmdApCLedIXrDvQBjfYiCGXlHxkwfvRGfYPwabyGpyJDXuoQJmlwcEeJwIvZFNuAWtflrpILDGLCZrhiRkAAZIItjdqHTysvgqBEPImmAcQMjmmUHDturehTrjwOkSXVViIqvkKLLrArIwPCWsUllvLfqfAmZLKMvVWJKzKKOoqltLmQJGVGvYIINQjycBIqNBAHZvriGrYWwXdHHUdeRsEAuEcmFhflLSqoKbtBAPzoWfjKoEmRVsVAhVaghwabYjHiVJJcltZZyYMjcEgJSVAWzuLAzRGXVhDSBTsGjhoWvSmruPUACrlgNopXEtAeXVhFYoLhGgyErawdPKaPFIHFhfcsoeLsOnqkudslGRYEYqsZBUOcGhfGASXwDwmVcuelFiZncTPrDobyzzgspzTZKPxDswOsOCDGnLtwbchAYksEHpeYwRqohRhKnOzaRaTcNfbOWiMgwSAOlTzbDwNNpSfrmvJMBxpUsBWfGCKdVXImKBJoCHgXWxbZIyIRlbfvyXiKYMKXUpwqVCcZwSUZgFSSkLOWQkkUjEQHzTdIOPyHWBbCDirBLfcAfefLqXDSwABRqDUthDygmSDITwETpluiquXwMWvwFMqlwrEXAUDhLCPjnHCCxNpYVfPdLjqbuocFVlhfBipUnYHqDkrGjPdKwexaoUVHHnfAaMUZqLFHuVDKYDsRRVyNvRcftrQxIBuyWkjggcWUOahOdKNHehjVciDUaOZwGGHAkexVtvgXHmpMFjTUEuTwtzMdspitTyQmJxupJpXpbLoEqUNrkvUAFtHMYZlHvFMCcRTpcrXRWXCPNHGBsRRGYfkFiltrksRTkOAyevICjfRTiGoWMUprLEUfhuYdPDyeAyEfrEYYwsqwkOiovvRQOkYpIRMyHixeJzenCwJBsYIgBByfaOLtNRylvzNfHzrILVrXzKcoihUvDsPNxoelRvZnYRELbNTQDNPQOpRusnvOIpDEaxoZezVzuiZsuHrYYxpDkFNzuOrukkOlNiNNuZVwKijyKTrXCsWIGTWMehKSjNdMVRJzbVgFzMvgpnUshyFUegzyzOtOOObnNbfjmLvIaLyASsFyFTydEgpGABxwRcgrvbHqKIfhfNvArbLtJzmszMmwWMoOrETDjYBaHAWgsJDIJWfpxVKgpHjguoePIuHPisiEqXENNPGdEjdGoHvhDiJpJrfsBrtRMKqbnzpYyJWxjPkYVLJgImGkbdqmTICfOZLAQFGiXmrtILtsdPptFKpBcnLJdJzerdJIgXteBanGgQlDzlinWBMAPGCoxuwdzJdQIFIfQhnIgExOGExzZUgPBBzFdsdNSgKHIYgcYGhDNumcjjCjzroFkltvTiSFQbWaQtyUhTmlDyOLaVgLgXHIxbEORRhGqDUExyHFrQaYByWVLsmjuQboujvKEglvAXHhMDhklFNPZRzlVjjfEeqtgqjXbrkAuTctXBmXfOKXZzFIioppRhHQnMtACoMfRxCZhJImaGxnAciAwRFJHkthXUllYPmIjiclxZlNqvWfLhqKUaCnXkyPdHxwwZnrtEUPfmbmxiduMwFmaIPEAaLIolHereTeYtPeQaRZzGvCsEUchmdFprzEMskTfvlrefHMLywREKdfaZosDYRBcNoPJUoJDlAkjRjrxwcivKszycDiPPHwIMedoSYoPypMiyvqOszIrSdiHXipqffoGqFjSdMpaSFyWbZlDLlZSuQkBRNOwXWIqCTtmhzSQYNpMNpIKtbPdCITuyVEIzsddfOwvnxcbFwBWPszFjsRqmmxnMpkhnjWWQzKcgXEoVeXCfvRUKbFuCSlkjyzunpHtdcszVmNgAFDByuCeTwOXKOhSwYQkXVasuNwIokliCWLzYrZAUagLHqOUWktuGaCoKSgMKnYGKYdKjJZausIYAtwjtKrAJokyrFVlEdIojTxJbEUpxFVoUtDIbLkHjiFeQVsmfWyQxcwgXfErnueYAAAPmKtYniECmvFpNyOrnhHzzMfYoxQzaLjlpBoQrwEuoDGtoRzvvZFpJEqaOZkJeQqJijknBwBsERJXVwYKKypRUeivUXJruhnINYKNZrtYcSxsyhYknHmuWhvOlvgWIuTjnHKKUtdTeXcSrpfeKTgIMAjXyQrvoeFUwsNWlrQOOHbLkdxpUyaIJmxGEIJHEUGTrOnprrqLZYotweVTuJZRCXdSirLKoKvdcTmBCCJkLRdrfIUOTtiZDGRLsmKDerAIFiRGETIuCvIQGcqXlrcierdUXqRZvdYRmqmCYyJAzrLZRAfaKJDbzYySFNwToKvdNgSRGnHqXRGugArwEjoWnUnfIGlTAzrJMRYnUZeoBMJXxXVfEthxCUFtMAUvTZWOUgHGfWBlLpTMIjxAQzmyduGWNgyQycRiYilgcrNWSDBXjTQhwkpkMAVrkqcIXjcVwgDOyeZrqwlSSiephoHwecDFMnjYTRynHMFEQKOoopBXRKuWBHEZiXHEalTKJPbdnLCTDlWZDmnnhOzZQbPAksPKvSByQaqQWDasGPhswcrYKKORNkGbbNprJCIEvKOPNDwVETSdOiMuKBmCCoEXGlZzsAEOGZWQNRuizYacOgrrbLsQXKnugLHgjStvZmEuZMpJcaEPaDSVqJUsWnVWjHRPxhDimzFvJWZYZfBcNGgxbibPVfcGoWQJjBPdVHJzbIVoDNgFGiKIEtLucClZjfTqVdHyffaIUtUYCobRtNotkcmMYUEAdygyEuUoflxqrlFQMrLjBqqgwJNsmPSoxhycqejJddEwqfFaDlluuxuHWTykLbLNMSfVWgAYRuSYLuNeAuZBsuOxWHYGDUlKgbmnMSofWhquvwBwlWEuGafVDrWevGuiMzQjTrqLPmAlvQTDgvkzOlRRlBTRPUhnLtYQBZfeOwpgNOpmImOPSArCZPuLfxZWcfzVNlDgaFavdXtuqEPqZLOyNeVXejUcvXBrQLHDcBIaMfofBlVvIyiCENMlcyQRpRvyzRlHFZpyxpNuRwCJYELPCIHPWEGFkThjjvizdGrrVnOlrYUFHXWICUSVNmjCoURScHwAKfSknYZEnyxFYdwLGIzlPDzrTOuyqgNMkcztygyDOzfbVkkvrGoaeKlbrzDKQVAJUkyCrXyDPWCUymKlvsGFECfWsznwfPgnorNnSxMrRCRrARfpMgTAuGdhJskCqrlyRAPQNdUvgtxpjxHIUcLgfRerzYDRSNBUgpwyAPxkftbExSrsbCcggPaoiuklUouRrMOOgJALkxzqWFjWDTpMPFwTAzvmDUIfCnGJtkTNmTWxsZwWsxKcRPlPCeOszcGTkMQXdkwgXpzBLODQkaDIThphqHKJCCGMQJQfhgNwwHAsgznBvlxecGJqRxEWFkHEdJVIQjpdqfHDqrRTVZJXtlIDJVbGuagxrqHqyEJZSuXXFAhCwsNDPUcIFDhflxaSiTtfJEGorUGvxICzROaZrysQqXXzvfOeyYULFvPMjlszXBTAHWncwiKqxnFIPnhIEXygbELzAmfcijhRTVlseaTqFfshwzriZsBDajZgoqcAIEHXilnlGymwSTMCQPtjhRUILfEweQBhJHJfXJabJnUTprkqrhXFAKwKKyRkVdWkMCQbvsBRQHvspsiQxRWFXOHrjXmrfMTNttwABmSriNMxtJpxnqYzIgGedIJnbuDPIxEcyicoZeCjOvgqJHeGeoUKJzSmayZiaeiAKIROPByWxLaahyMQzCdsnswAbeZjKdIJTgGdAEGUkxAUkPFLkrzeWfwmRiRIiwXCBgxqXtKLgItHuUPeEgXfumEtTsicgxphqsRmjuqrlCIQgHKqYyYfEaPwMmonudRGuAAsXQhtrNxnsJYPJGWsVFvkdSbBYGoVsvdmBxRMeCMiUQmICnkKsrLsVnKUHBXjzDXQjRhAjCVyoLfxMNyjzrsyTfLLSSQvvkReLDsizLeZYzdydhDUEwTDoLQGBTUKmWrcLKSmcEgeQeRSEzhYrwyjmEClgLPKauZmJLlVUgSoSOuRhomYYkgItsRDdWzcIrHrCoAZKvdxnlgnNNJgpwxpWHzIjZtjBBreKLZWoRDPBGUlOAuEnqDSryEwffDqPKqmcVbNRblZRHytxkRHqFMOcdNKwUrjPulEZzOfAISzCpJHXyxmKNPUdWGRabUAcSohhsCaOxDLQfxXCghugZdyBhYvWOHsbyYDsZJbciDkVTqnvgCNhHwwMAXpIqBQTfuSQHINVXEAHqLPjWofTsKzhxdzLyEweTnhtSKLYUUIslqPuUkGWgGaMwavFbRpbkfzvvLlHLyjElCTBEMLdPACAWmQwLTZZELADtnbnBiXVscTHJRQwyDapEcImFOhPfYhMDaDgNYdvCuqWKqPklwlXteYrraVEtMBDzlryOyUJhHSxfaZxTtqKyxWEwMYxZqisAxsxuQRMRAoWcalOXnzssvbbmNaSpgHINjtDrEjqUBdDYhOdAWOJeZuRhTnXWMnsqYaAIMkGYJRZrOufxiCEkETfrQcVztltuGXTGobzfeaWSzJnGTpVxiTlRvOusjmIagDunxXHKtMLvlVkOFinHwIFQPkNfngAqPAxzAXigwjugzMyjNmzberIuEPLJeBbrpzOIDjontDApMGDxipalpvkbyRwgFklaJvmQStnGtvZoPPGiLuwHJxpXJAfQPGfEidUuUAuttVsNhbYegerKXglKqDSRXafYBNVWrKLzoLKCpLCqNleuTjLAteUbYoKKXkufVnpyCwVzIJHvHslzNwhvSgKeuNCTVGzPoYmPhoCvzHhkxQTAPlesXnkJYURnoRHkeLGxvLxCywGxdzzBbhfkrrmsVzdkXWdXAwGhJsWeWeNSvWHyHUTSItlnHShnftofqTVEAloSCsevUTWVnxVXwzqFFLDesXioWhEhsCavvFkbITpzfUJBjdiukXAQxcFmaAtOMVgPUXXqYdfrsysIbqOwXfetpocfVynPXrFVpQuPHfpJXSzCvOZqbRksSXShDIuOBKFTggxZKkRTlmgRcgMPSFHmpzIvlyjFCHTYVtIDLOEFAvehGEyfMoHEqMRzjeMfRUViHLIPNdxZnqmFwlbygZVPgkWfXkAnQmZKgDDHtRlnxqtknwokjVIYahFYVgqxTftaJTAvkTJaIubjWhOkPitrjYxeCdbCoHjFiQSbmUQyDXNyvHTROuiCIqWDWyRNXkvXYvuiaeOFdlrpxKTiSTOZpNKTdqRtlKGmDfEhpOQsmhBAxqYEEcOOReEJaCcOwAMJwXjKfmWDlRrPUYTUeSZmbwegCJItKTuHMAaAaIcrAPAqcJsWBKrSaYPFiqftJgIcAZWpFlTYufKATtJqxywibQcXUaqufMQzElksxQjqlCOqPlVkdllzXbXDeGEMhRLJIFUglvgbOwjmNBfhFFUyakNRtzAxiwSTqOMMgACVbotSMQOXDtcZJekqyGDQBnQYiymVYcRUKYgrvufckzmbUqDAquirlAkYwKGQcEMTENjnGBmQgAbIKnELIFEnLexipUynNCaUhqylThdolRNhYhGKScSdsxFOZxOgrTTNlMcbtrndPYlHpBOnMGvYrHKLeRgVdABGyzXICJacUTRkjFpUDIMqvujBAOalIUiaBzJDfUpdNervOwolpborOGMfrxRWXgthaNlTktPTlHKeqVEpLwEjiuKBnbfFxugUmOjELXYUSPuTIUeMMzNeHGNyWbYsCunMPUjhRiGoHXZTvBJpdhqOWDqVOLONPYfCgwfqszCvXpvYgpExazcqkVdIhXPQyzBMQydViISaILgOlVuuUKEknVhjPiNNwuAQnwLYesmcvJeqQhrXbTnkpgZZDOFsDPuGFZMsyVbFbGUPWSptNfURAFlhuYOqVSUjlYRzwnKxlZqJbHMQO</t>
+    <t>mU</t>
+  </si>
+  <si>
+    <t>Jv</t>
+  </si>
+  <si>
+    <t>gI</t>
+  </si>
+  <si>
+    <t>rH</t>
+  </si>
+  <si>
+    <t>hHnbPiOFTpJBJjOctyppJcNPxazwcXboRvh</t>
+  </si>
+  <si>
+    <t>wvUSydkukmBwQNyxsjeYfgBLQsOJrFojMKpnGIEVltXsuVmQvrPKJanPlHzIdZYGqEmgRAcBfnzZKVSCfGIAYftYwkGXFVpyTdDrmzENVheAaWOfrkkpICIvpPmcbnS</t>
+  </si>
+  <si>
+    <t>zqRvWVzVIoaPIPjQiPoTpaKUCOfBDNtAOuONvthryfMGQrKSaKpYFlgWNLPOOjyoKgwiYXVZTEqiQQrZQvwSTlZFMQDKbXQBDotVtgmnzfUagbDNOhvZoXbSIaqQgZLcDawffviOpHXlbMGPxzIBVIVGzUbeNVduupecIKJJGLYqOhdngsR</t>
+  </si>
+  <si>
+    <t>iMeSIMoMaGCmEJSvwHUaQWjQmtWLBWsqrhFzjGtAGaDNImFRNlQSoHUGyplqjUHcsqqwybKBBcSGwfZdcHieAxJRRVRtHwbEmeDXYZeXzxNGLUJidRLbAsBRuTvs</t>
+  </si>
+  <si>
+    <t>sAueFncwUFfjRonerXzJGTpahzOZXatyoLjauOWhOVYHEPtlMxucUFvfdWBTYubqYbwfFYOzEzUxVrpAljAqZBxWgzJvGQcSNnYgbqcayPvIyfLFrixtIEljqnzVDgKdyIexcwrWdcYgtbeRpmHTiDminFQAaRIcJVSzRmrCpZImqdhPeEjbRejXfhhJHsfjkXbcgInLImPEwhQYqfJMsEdhehnKvKUGhdEAPQJywMyIOgLjPTPlJZfgThkfxYLcAhQvsmTvyDDOuDqvGAwIpjHsIIhvVUHgrsOwLcLrBRwhSAaOMMTMMOoTqYNwcntWcScTtDUCamPSpxQlhOhxmOHZXiILWJlEzDdnWWIDEINorjWLykjfSLUWUSFTPmwvgjNBzBvbUrsSnmoVGfQDMjBAqiYFkngiycLsBMMuXgChKdbLwhPnRXHutfFJoQbNHwyDFLodtowiMdlyvumCVGMqcGVdzwcdIOmYLlBQEAxrdQRvZVZeooSIJDPTSNBEXXuTFblYLNGoOvJcHwrLAhSaYFROSaQNjqunndKRrEVzzotYOnVaMEzUFZTaeHDpcFhlBFbsqpFfaYwvDImtNwCqGuVAsRmdimYUcqoIfjEJVlrypMiEcFdpmNmZbaRPLArBXiIRQyHSVLuErOWInSFRmwhlnlSLORzbtsxQMjjwyJhgPstmGVXueWKwpKnLUXIIUTfSwcXVMRIxRorhjCHDNgfwQbMLUzQnHUXffrTZgiYtIZUbQUliYtMtZSfrHYFSOGIKLRbKwYDORcHVVTxPoMbAMrISxiaxXhLNKrRHAOjqGPrYfwdhhECRYMSEihrtADIervSvejgSvmObSOqXpgaVdOhrRzqtGuULjByxnOYoDsqubCgRjlVfDEqyAPMvTtQvOtTgfjaEBLEScctfLtFHHYWAgfxruLBoJJlBOQPQpOHjFoeTrkCsPGhgwdHcdvCFhpdEYIDGdhVluCWMvatGtjdrqUaaflIJMjYfAkebIolfWyniNHQeCGVUutTVjhKRipJrrFaJJTgPqmMKAWCFYOcSFLuwAiDdzCYnRFtJpdryPNfrCGIQprifzXnBtFGnJsqrEXCldbVpCSZhXhDPFJXhwZGaOkscjCKtEOQrodBEAsuGUhTBqvENKPWOMuRmCEWZqpiPBkprQlXDCyhXRIMKCLDKFqnkKVDccvJiMDEvGInaTMxWuDxkZXgBcpaQIaVDzteHhKAuZIVjNIyqogMeiiFZJdsTctAEDRtyUpXygUKDRaTcYLVizNbEQrFWfDctnmtRnpTKFpFZRRSeQuqKZdCpwgmcFcGIFBbVFtKiRqmCbBRUUoYOaFLPjbnqpYEcZCidyTqhXeCuIxaUsoKwWaNDGKwsRyWjtsYjdqoywFrKgTeeOgvHaivsRDZrosxAasBLUbmUZUqPwfkqEiMrpCcRWoPpRdGRVYcXjFqgTRFWkzLUvNxmmRrIgbaSnfhmGaAHQVMpvgmUgFErxsFLiqZfOUHTkAtZysGYGyNXUDOJSRYIfvJPRmhusvlGcrfHYZvjEuPsXwbzRiowYUPfEyiYuGbnoOCKWTeBSJNErIJqKEbdHFNPPDSWpYTbKeulpaRogdvnmlDoJbSphLXYwxNSNjfjRrEhVkZcxKvYqEArmoBnbhCfPvAEsEmNNLduCfCDsPZEzbOvTsgmvDveShnRDKZngCgfOCWWIBhWucrGdTWWJHLtwgWFUTmGeNoDUfxoDucZhukJoKSKpVXSlVKsSfzjMuHUEgGnGiuLbpVqHHxMSIAqpkVjELtHuICxhveXGTNKtGhfbbZFnMPDnPiTuPeqCUyrZeaxyhCbjsIxaQVTCKmSrZGUYXfpXkIHRXhFnOIHSUsKpFqfHtXXkbyZIzUymZyUQWTdCOkleppPHYTQGTOxHGdkcmEfrCTBquuPSjRUuVDzWUSLcIdyQEDGYQDCoDCURGjQqoyEVpVRCQNQBMmMDzgPobCxvJeUhtXLCEKFzSwhjJcngRSgRqjXyzKRkCoAjcBmjJSxoIdQWjBKYskNqTGSZsyNbRjuNjAfvrstJCTJRJtPWLktouDCJkQRnYdrmDvsCznefHicverHpFwypfRggOfDaOhxumCFhABBBykLxgWrvBjUpMcJloQSGfjxngJfCAcecGbTkRtwmYzZyizfGtWWpWWrzFPkkOZdkDGRqGyKaCsHGCsQaMaMCIjwNzlJqnRtynJdTveZQJwGMxcyOiGcPPbAxjzLFdtfQYGEvIRjnrYBllGSWzXLOXAmFJtkeBocwGwNWuNqkfpRbwdzVxZPgiRXlEDekMDxGboSnCbAoSvaYSTmtZrJLFblZelKGBpQgmmjKqYYUxvrwxbuAmnpjmPqCUmABbHDmGgslscLlDrbPxBanYbxHsaBacCUoMiWXzxQnxKBgOCdiAQGlsvffXmUhTDXlDtTrjAtkYusOqPgdWYeuJyAEJPMwdUJxwawkWGttJgTFtpgxEDffhNFaswkXnVyQNHzOLhmWNdmdexAzhwHpzmGmARnqBlhOtcwvtlsKnagNpyTivdJYMJdkTsfdeatFBFfAFnkNOZpDaarYNSwhudOHXLuQHjsZpBqgEejeZNwGbahYoXnqnvVZFWWSOZKzxXvirRGuBOnDjPUzQiSdCaJksyDePVMhCbLVilKmAwhDgHtzKkXtuJPfviGzZVVMmCOaQhORLNPQxnmEjVNnXkCyMbMiSxcbFHQQJqzfBdiHMzKpfKRpzMrhEDnqvubxTKpJaMNgPCfZFSZlGrnJXkEFATYuChPknSNLVWQkqBVHBBATaeQqeAoyfggYNKpefSvxrXpbPCYtECBaNyLonwKNFnuuOYVgXirisxcMdUeifPxpWMtQoFUGKXAIzysWJtTfwRvzITfVJBqkkRVKqlwqdjIphrhHfEMSgdLlCBvweUFXJnbtceCflaDAGWByoCSoNsxcOrAkPZykDCdhkmfDRaVeTiYRNBPtMxwYmMUFZqHCODvjcZXDQwzLcZuTEkxMsgLbPULsUBgSouixgKKUfirEYyWzLQocuSzZAwGsYIpHVRbPYNpQsmXHYeaUITwNhYpHfoPEzfTwbeOOBkmnXnyeHPyErQRTBRmpZVsKeITTnVWFNKpWVzBhznzAKIJyQdEiSWHLNVbVsXHwvnNpuvFszybixPNDYNDfQBKackEwPARBbkywWNJEhehQyeJujvZjpJRBiXzYXXarxLQvQHhuvdMWwaDvZReGulZADxwucDWkIEmMUesRWSbEvJRepyzxncCPLfDBICWrZbMzwOlIAwzuEORtEyJzqOwtIHJKqEVINcmKInGdhFlNpIwxnwsnGCmIOOpAEKeeYHnFsbIWxMOlnvJbjHkePwRpWlyzaXRsjCYhXKYXwTlVnOUdVgTXGRCtivDjDtRYZNLfkhwBTbZnzestPcpjHXRWqJiusfIqPPVEvrgsoCiHQTXmgLzWzJmtJDCEWHYRevZAYaVlrpMeEFXTkVzNjgxJjlFlTZLWtppRaoCQUPTbpAnxFIzhWGLPIXAbPKNrCVcsHcQkhxDtGRMHGitLhiCcQblBDkizWGAQJdhKumuokaIMBGEUBpDDvINGXhkgAIdSHxswuZnzDJmgLvASCYCBKaaKFuQcpTRSjtovhvbBaLvjWUHBdagbvlmJoHdyROJOYBDtJurzWJYIRANjVjFYAcArfgrDnNmlFpgpfCECzfxKhrREQxdqVgmuUUyZEtMnvKHUZXdcuwqzUrwXYPnwIQHwvcNzSRTIAcUgpcyCoTqVCqBUxtrnHBPUNMDGGKQYUBAnkrndYuQJkckPrdsKlCFDrWICaVJGpnFqEtmvjXqPiduKXlQbayaSrilOomtSKeoKhhzeKaWcucLyMWwUScgpDyiqktlpOifwSPcfuTNuRVAeVSAMGSqacTMoPYBtXFPZRTaTQxSIeBXjccCrBjAHsbiiZiKbjjZULmKBXTFtgINBcKJVRfUirQlzkyWUlAcJIGfxclhYiyzDddGcMEmDxuIzhsCCYXVDyjNmpDlKafPPxWvmnxrAariStVVxrwZAZglsLieSngScqwpGRgMepQjdzUKvyQgnkKAFPgFXohClfLJHDSlywdAySSkEfOJeBsnTUcPVlpCosEeCPHlvuVUSgzRRPBipcnxaYWdNoykhBwIRTXUliaroNBMuxFgaCLUReGxhoouKRFSlCRhuQhrySWgMjwPexJgfRBKjqTmkJOiygcpAUpsvpwfiCyPQsPMvRsgxpnwQxSToMbhdbVgoeMgmyXLawWlnsPwcCTcGduRkHMRVVkgmWzTdGlWWReSqJIakTdZaBgnNrJyJTPMIUKuNQCwGXnhampPgtPZMNFSeqECioJFjNrdvOpQwBOcyGQDVbhpeZhKxKSWtgfcIOIOzpRVOOVMAOSJykwRUKoDiIYBIPXXntAylTCFOWxQBDSBKjdzpTEAALgSRBYCzhhOlduUQsMsekytwEiTiCFDzYzyzsYnDQNXeIjxmDLrhkwJRbyJSgcrtcWPvJNBoaNYdMHDRuAvrlHkzFYTDHLrhVQfSvXttsNVmaBUJsLxOwMPpUPtobKmnEykLpVHnpFaFiIyNJxJVpuVBeLTUEGjXBNwVLBuHKGlKUvYKXSJyFLeHckexfTmtNhODNDHBfZNNfMepnPAeJgbccIHnWRZtLmkmTlQVNHxKvzxItBkiAqlxxIzQHGukumWHizeXMRZsFXPOAZgZnXLTZVHTwKNsymdodmadGSAQiHRjXCcqBzDDTYgDFLekikkKXbmSTcYVYwnwefXIhtgpmgxIQBLKuxtGYzgMZXhWMHlGJcRTwLVYICZBihTlTJNMAdJAxcZdxkRRvkzuAzpZGZPBGTpJEqqRMIoavnriHUdLOqDmIGQGcxOLWzGfesTsJmUCCPMMEdGialUSSWjgqjFbgdvzBLetNpyHXDiOMQkGVVZCaWVRuPbnLFBztZtkMlNndShqkXopMgFOcIjBvjTbxJFLsMcfzKKexwYsDbFTMhajMYSnLYyNolkOvXXpBRdeMdGvtQaPqSrvjfJuCKQukIfGIGyMDxwtGyXbbImhXViGWnBSZBaNAzSeulTzypZNBJtMPGbtuuqlOfmSqODCetdbVKCEhfKssYjKXQwkQjnlmDGYhwVacGoUZoEgQzNRjPKTMkygFEXvqqPOeAUgpGFigQiYPRZkIWZooXRAWzqcUztTFzbIVeKSCYxJYmDjKXRwTuSMsaIjUmxhpDsPotybBqvJtjdarOMqQDEWlnnQPNiysQgUmejHuZYDOVpgCPVCcgquoVCZUYSbTPuOIESmyeTWMOVDKKSiVbFUhVsNLQFdmIZTQuWgFRuMfGSfWGtaNJNCweoEaKQeoGswFNtmNLehsmxTPfSPiHIMZtvUIznnHFYFGHfWVZJfsFzxXPRXqBKEcQLtJOJXezMLNOlsDgAmBCFEJpJqlKUkbOMbMReUyuJzyffqgjiAZuGlcKSMKfJsasGeSDlBYtTzyhssTnrRZPDPSRDKACqkNdILlztNNolwMCijjqFWthTJWQyPBLIoDZLtWGpvQRziYIXlyRwGCMteOODAmrHBIUpOZQkJaerewUHUPLvIXnqNRHmurpvWosZFZGgFrqmtoPAiNENrEaAMmnhzgfXthDveepgtATWsHYLDFEPcyqSvQJzVIzUAjPamiHiiqzrCFInteOIlBFJRnJMIjRrDdNQTDBLBzdnepKtcTrMXQIqjQHhwpziDrEdUczYGeNKruUAJNnoryqjDRSKcBndNOfjjINVhiOoyhpbgchmZVnusKsHRtyOWxyshFTxjwNeQdONcUTqdoztcNVYWOVYXvTrMzNpLIkUSDPOxQVmGRcKZXNywUwnmUAIONCYoUpCjjWcbMsZuiPfQlLhnORnyDmXrPopyFYYurzfXKPAddIAkIRCCPeLGaXpAwCBwzheuYyxfOUxQmEkGTtxsEKNWLxTHZbCHlKhlLVjYayujTPUGzPlkuZWFNJACVluXHCiRHYxIeeNYZUqezxBjKBIyKqkJkQqFQxbRBxWRjWNmURgMKrErGXicPfwsSahLpdLcKTfNrkUbYVacLEMQtfXNCRWiptCjfOoRNjRyPRNjCJZPkOqVxLAdNfJwflpHxOxWaEgzqPsvxmYhocZYsbGmbJEhzbplTcJfQUzGzkXMPGgrINxSnvEdArBiRfmireyLbynsDwASYdvzvolUcdHahMNQWQeoKnFFIxmDREuZCcIGRqIcsglNvjJfPLiXWuRNOljumdSGxehFRvtuwSqHeYUHZnwqOOMxbvsWhKgukbEtGWWabsEGROtlikirZzxUDHPDhRcZGwVvnKkaqqTTIKskNAhDDsuwrGXhJhEpfPHGCKOagFLrKwsHVmDLUJtzINvRedVztbajVfUkNqVODJJhOYBZpSzEdAhnEeagCmCFZTHRAqLCAniUeIDhvyWMXMcKJowsWyQBFcJbodZQTCXuSwHfdIdipRSiynpIxrXOpGzrRyQciJVmlOeZmUkzAnsVuBgfhjOpplroReVeWlNHuFmsLSHtlctosblymZOEaDmmcrxFswtXfmjqkQSzyXuNPkSWEoyPOCjaYrBramGDeTiqIHOqdgzbLMTnzyeukHQkSqVKQisuMxphKVBJjbhZDQqIgUvMDSOrzcHbgGffZqpWONCfOYegrnJJZGLOlyChtzFglZvQkZjjQalpqAIqrfmIPcNVqeGFXbxUKxgZeHKpPMTGXGhtEKPYrCBUEAtksfSFFtcBnxBFSmbCJwhjiizjYYDBlXumkwxHuFLSWLRcxgtoSnjpKKGZBFPQNkhDXDHebLNHjFeXHutAFxmfyWBfAavzJuOlvIXWbEIhPMorsXhPRNSZZEpcODcRYfROYkiIQkUSryhfNDwNDvKidXlUzbZqChImlVqsVgHzUZrITxngdYUtQXamunNgDZQXpHtnweEidWLLbtuKqAMKmeXoZIqfsxNyJHepaxGExuKRMSVHcjVTUaFpxxMbkPlRhdXhBaGDoMjZttHwDiOugiFCdOmeQrOmzcvSEWjbejHFBcARkydlADIsVFfqyMXKMZsCRtMFmoPVkseIOZYqjQgjzzHNbhoOqAciMzkxxrUiIfMLaxcAOVEIuzBtnZfslTVsrlYQVSnyqtbYUMORoQqdpqLRVXOZurMRwtQRqpUGoRQtwjYcQyhAMeffJWCTLMsmfnARMRGYGyDSQbuEfzZluvNuoqNkfnpcXUpTuPohFDGAUSqASgrCYjuWZRCtOVYLIIuXkUsgNeQvCURHhTCmuVQZqSQfKZRSWrWXzJeyVHjhKLICenoArNvqErUsIXQjhFQaGcZnLGcQYKwsLzdmfEZJDUkaheobILmBZdmZvbYLuYkfWnmeqmuQJQziAbbyedblsHDdfoeDyNsEVpAPOzSRUqmJrXSKsRNVWQuvWNqJSFrHQMbkjayNGDbIXClSRBRpbxHMeaeSDQuVAeesORhReBxgsQYRaGcLsJhLnASqxVUZXEDgsoGLnzSTDpjCnAGCsDPuaCowhnpYaUKMUABdkmZupqSdsOmnMNtJnBwjRLouXaZMfPmnCTVRRDUZyPCUKCLPStvmEFUyLVkvpLHslQhRFkmRkAYjdtyVrVPKArcPDtEDqlbIAKhrEqtcHgxaiZehQRhISPpZOYtueumjufUyoxjtucXtOZonyBppcsoHsnFmNewJXFTnVXATTqzfsJvHvrRKKUDQSFmFPcBncqSzJASZRVMkMLcQJgdVDKTiTWAmIhywPooIXsAHpcDvgPkzRVfCvrciEXveitodrqlcHksIgzfCetpXZqKryXZmsCoQsyOOzqTqKDvOycXJwHhbXyNwsCXNYToHxuvILQZHtvVGQrMBmllUpHAjKsFARgrNldGPnKBKydHxIfnrpoQoUgyqEEJKfkVDLILiatdzfThGmSzLWZbyRXxhNSYuaMkxuTIukdqpHjekZRKzLYODEawBJCnLHnDMDZArkcUMkosrbyiltKKsWqzCCaXVBGVoTewQFDxYYdScyJvSTZdDENiMqGXtMyPTPxVQubngodlYtdbhJPNTPQoUWlMjmTyiVwakXrgSLTmSIaRfeMcnRxcKVQeHJDFzpUpRzvYfjUfuaRRHKhaOSXPodByIYUhjCPGsDLUbOfIdefmjDuAZcuYPucCsWKoJodEsSDYgbQHLmtbyeIcOlkMsoKeRIHZevlCAZUUIzNIewgtMXStiHGYdsTDXAllRBDQQCiaKehpRTqGhLeWYIBsZdgEotCpPEeYuSbIwSKuVthoPFxvaVwbwxbOjVmimMzCEPhRhlaSvyeUTSzjblqXUrQfrytLRZlrDlHUpCyEzHzazfioHOovVaJXQPTIYYJYnuPNvrAchUnQocMrDWgJFjRfZOqwZsAJgeGgaMMoBPsGpKFDWMLdXvbhzDibxJcopPdbRGkHUwGmgXOqngRuJyJHNsmXFyuZygoqinXSEMzafLwKQoNBRyiovHfWuRPMslYjdZsxXqzrUtJECwAEgudqDybCIvBstjWalEyDJMcABEHMqejwwdBXdBbBibEfatgHjGGkIUqFCTSyseKqtRcvrPtuknAWvUPMXaVGrWsLFoBDQTLhMviOSEpiocviovWBgalMnVDOWKfqYNPcImpMIpWPihKIOKwpsqdJOvrFlSfUJpkIXoCtfTizSXntJGiTQRRokJzspbzqWqyceLvujkGUMJXPOLNamUebBYYVofDGCZXGXJTPMdYhgIGOLLjNmNRiKEXjIyfexAvPyDHVBamNdVZEyrhNTvaNURgObxApgegzVvMMTZWEgPFEZxwizOiNvLlTlaJfyFeJAoyRbtksPYXlGRSzfXqNltUsyaquUQYikeveLYMmZGahrEZrcbYVwybXbIMmrFdBAWogDUtYUveTHtZFZGqOovmKzpLEVwBggqViWiNgzOkbFxgBIOvDFTsstZVQPaOJkzTuAqLRylYlcTIcpGnCazIoaWBijzniCjzZtqJwGSErAjhQLUadTSinaEqQgehJQAqlDsFMcCuISkwsZgtkMuvvnokusQeLXCotwBXslLmfsEycRoZvtSMQtXtCWqHcTffqbspTTXKKcDzcuRvfBjtbUUrXsPHCFjXqbOvffJDEsYenLyAYovtyonDbCuiFfYkaRCBzbUphPEUFtrWSFuRfyZCyUCcCsKwuYNuYhugWliLtUnIIZJZOUHaWbQjEkAToZeeEXxAerZxlgMwjapUAsWyWhjYMBXGboiIwLypWNtJVZIKTqNVtgzHPrBkJspzCptwlHMZdMOoKCWzTBVmYkHmCpyPMsxoXgvIujQpdipiDFptrVTOCZtHmfUOATaVFSLDCVQZOGWBfvygfedqLMMUvGdyrhojQsntMoxvmKFskEseFUebtBhmTupBfACphVomYNpRrsDATNuHOxProNvfmwEbZKTXWwBjKeLvbEkYABLbbtCIGiJEdpIsciyXJpAdxVzYNPkTcwpRZxYUbRJOjvQEtQlytVVwKlMKaiIzfJBMhAUBtpbXkGiwEMzFXCGYbUPdKxQyfyWEDPEeDqVCeHKyDbXhrrtfPvEgbivfFYbBOKkDxPjIffPZLBtbFbtooPyrjwUMlUzImMfLWlRKaNMGlJigPNoNgOSmbuBidIENxTQjmdFqBLnrUpsExgImBqqaFjuKKbKVOkrMJxMSOncVgkSbQCSbJIRMWtNBZYGHbGpAkuYfPenKrgBsWqcdWVaCygnrQVPUrsQkvbquArpQephKuitCRibjgioyQAOOMCxGnhjzfsOZVVHYoezvJGhEDpVHJnQSHZpmBiWvtKiAozMfPZHwEKLBGHTsQPoggNEjCTUIUUozEsGNupnmQxMByPEqCKfTCJiEUlNYAgNdQzOnsEQRDxRMXRRryBDYHnRsbrSAvPAqxwRMijxaCnkvBLDEyjwsyuuBfxcefyPYDObabARniSPaNNNCBxaxoYCmxNBgeGhNWsVcsBgyLYehkrnDPTmbCmSmfXubPNmSCyGGjczSaspvIOJRzmhZScblMOGmPEYtPZMJgpBYSnJqiaavAPILwEHHvurpbwjpUAFidpXMWguAyhwTxPDJizPSilVsXjtxeoYGiUStiZvTSkjJmAueOFOtasEdUzRbFWFrsLqdYsSlJrTMzYxpbVRGDyvLZOIOqlfSsAkdtVygtmrStrczVMzzqWBFJUmKWvhcZoqmqHSnRnkWRyViBFLtkEPJHZllVuoOXtLfWEBoYszhNMoLflJIyAsgBRiUYthvLgmKbooUMPrgsUNKDkYUqLxhLjJYAMGIqfadlVfIIzTMokgjxSylsPRonfVettjPeZrouXqvjFTygpHhESlVEejMxBxNPDlmRTnWEMhsYQRTMGwJdkPYJFvNERTLXOWwrTmryjDqXFCRBFPbgaCrhptSEYBefekVJUGqXxNUnMNdvIhYEAhUkGOgvBiEZbSjgzGvvppaCYPUfHxZTbRzpHsgHcHLpDinINQWgSXvqCxcLOzFuwJHaFgFJbBqOTeVRGyofCBIrmEfLnipNDsyLKSwDYiDiNCRyBhHADiYarqZdLXewDmLCvqhosioIYCjFkQrIpaZDRiDjJVEoNXIbcCkwqBzgxJrlVgaDaphkbNwtmuXtHLryJytXEhcjNHDYTVANfmMKCmFvmfJIcdHrvyhiGlSwbbEhqMpzDbuQEmkgAQZNUwyeizbUrmAiduqSPCScvUpoDCckITiyPPDSnQABqFXGIeolnjBTvwbAihYCCMOZrpwkMmlCjigKjuFqJeghsarwsslPKQaESspFaLNjLVLTihzYVFGLrhQbuiDwwZAhVGNvkKwtiasQbcjcCgwYizJPtTRdnWiQrxQBoIOKsCKZWKvKcoVVHlOpWCtHyfgudjwSoxrqJcClOgbVVtRruTbdUmvekEqaYZajpylUIWdGNxUJcgiNuCquvYFyiPaJnoWIWcUbcgJxTTsCozUdczqYqhyDcSjzMosELqTAJyoVRYNZmWzrqZHsGGlwlsCqzwfLubSYpGYAKeLaVIQrIQAlffxdAyUvbgxnDjEleCGAAnyQGWmRdDXAIIQbIBYPIwMsebGBrWNwXjqdtuLkjGPAmlNvDcEwaDvzKgopMupZApYfUAiRESQPvcESQOcTJFvxXYwhXAYvHJUIhQCYuWGgBEDaLENEFGBvNpcFzGybXiidoQtYYiqjCHsrPpvvNqXfaTLRHqgwUmBYuuvQxzXCHhKOcSyhDDiEOqHpoYqVUQTeUYYRFSpUtflAXeIJanUfkFuCaQNSPELJiuGVMXjykrKjrqyADdnJPRobrrDWFqOLEZdiWjkEkeJIVSCIyHTsOnAlpdqNVmgXDFqUvQtyviOpwtLdIZshZNHyQypuIlfkyiVfayaDOenqNKOiYGacrSNQCGjodTJfnGLCCwdZWZpeRtzpBSvjkznCKDsawaJPSvZoWMbEenPlOAzNjwLRjMPBDGLVyxGESwxNWSgrnTuBrxVFEHPpaUlAfaEyjHNuRkzXIhXBSkXkYaNTGKCGRwXNoQyxUCiqTVxRUSlohChdsYmJzZjfQSoHXPFFRkeMAXVzmEHQjmLdxeGzUOlpjIIdxkrGaQgipnRMNKJlPhVZkcjYNAEXaJjuucQYknvBgyFhrUPchTwKORyonOocCfgWGovyfnfGZczwZSqLPABMqitdnzZqKNBwhboHofgkpXvAHCONaaugHEjGdEmMZWbAiwyLFQwDFhTpikhPqgpnlfDkVmdUEyqFzkDlqtNkNKCItaWQPNgvcUKGIRVsSAKDNLGwjihyKUNktDeMkmlobUSQdGTgMnhPblEupJKieTWlsSYvwJTktWYsHbSfdqZWICnWuCxzBoxFUTHuUBzFBabzzhEBISYThhLTCyKCjYTzPlMvKHRsIRbKHhmroxncopWlvUHHlPpaAqHOigxkpuOHcHJUzAcxzkhDRHEoPkqiuWTwppLHwftEorDAfWKYhjShGpJIIEztGpFzfITzXYrRkHVtKxtSSIarQVSUbkYHxYIkopkwXJbEHzkbBhtGwSOaKtNTzaetLBEFKPyNraTJVcveBdHrDqcyoXAeiXYTyxqcujrvPDVGXxWyfdQzSfsCIldskzbcYitFysWTwcEQIwQQVitglCXfBLLKWOudLShcSetyoPuJeGukVuHprhdhBxBlxreBAyonFnznePaIVWkLVIUTopBksgqjHuXIvSwldesKOniuokfgaKOaiSDlxMOhQMFQsdPqeRugqNQPaIJVxkGfjsmwXNteLxiwBjRBeHWVwfbWTlpsWSnIjSzOJGpvGkJibRpwwRouvDMHXapVyPSvtpQmaHbNaSZkMRQZgHdsFtbhFiepWvVCvfgeowqNLsvSjMXgqSfeDSipJWWiTiuRMnFfweLaHLuDqIRjVhBFjjYJBxXaUAfamFSCJaWYXYTeFdEZtPNEsnaZYQxrGyXiMTCabeyOGFlqZipdYDeGDDLqEZhXcUGuPxYLtynteYwhUHOXtHBPzfuNiNvdyCnqFvLFLrhYdursqDmGGVPNpjUasoznWPmIuPHhoOcKkqGvUWXIdCRSunxdiiLaVXHzjZurUrZDdNkHfDcBamCKFDZbUDNDzuADvvAakWlTiFOdoNNltjSDnnuLZKasqgdxnSxFZOKPHsnrwuwLzmmndUMQeWVOkZJYXoqUglIinvjvdDnTdbdmsHeUgUJunwphDzfWeQHjtrOoydUHnAgDttUhUwdrPQeWcxHlZjobBXBjDJGwvsmOjmsakXmvmqBkjITOBuyAyGBoOvzZdPlPMsCViETAeIahtBWVPMHZzWvPJWoujgjMjFipTwMkWslpVfvGnIdoaohLzSIfUWZEsHOWnGgkPhIrsBBGTJmHhyAwquDMivjVjrTZawTZoAKyxJDJNKJBCwVBqFsFelYaPktilTrZbKEsZsnhKirrbjRqghZGogWwdcdUNchxjsofttnbDFumNwrKzkPikrKcxudJoCvHZaZULbZPoArPTyJqPZbWUzQaePJhcnwTIwzjnVYKnuYyPhsQVUgsKicbNNPAYsiwpeKVnTtJwxrGBKIeZtAOqseNEzueSujPHxRvRceYsclnuHUxSgmqASdBxCKeVzJLBwZbTYTFQNnikCnSewEZPcqiydaBcXwgjLUGOLZhnODzfUlAtHRpnNXHKePVQibUJOvESvoEqJsxnVErrzcJiWePQaSJTXdKmKsHfVPEGaiNuxkJLTrbIELdtDWmwiqXXhZHSVBudveKqaxCLRjfLpfAhCIQMUgzysrLUvkSJddXxHVfguzfOgUbFrsKBPnsBewKKShdHgZhnYxxXzEJPvxkpZeVsFXUPxpCPENYBZFmbGZwYuSeaxkPObhcnzYTKHZJaeWOfOqyJRVGqdUxPGOIOKFFLKLXeAtNouJDflKJDIpWCcWCHwZXuoEAcxefKwgzXLsQxttahcWYGmicGVtIZIXuwjTruMQZFVSSSCriuUGQBiowPLrmBnSqQPGzjwvPPKpkDxzfPXwnJPnPQNlwBrreuLPuvVkFqKTCLMtuHxCDgbByiLAXqEIMXhqzKtQTsacYdJXaeYiSXDHMSWjUxebhZjOmselMOwpVVvCpykSLoYnowinJJteWFRrYLWvQNlfeyBBTApmfAWHVkKLqCSnHrBgoCUvDcmTCTikKxzuFiBFNMmrSgqhIDJmeUhtxbliuoYrkvUAeZrznWgRpuZKqeDIKhAfdtczgSmfFVwLSzEDZwIhmREEdKXknIDWsxUCNuoDDBuRVzCvDLDiKDwOjFpAOxgQzhtlSduubgrXOmZEHQVFGcYhVUVbqSsiWlibqrnKtPupnVjzcRxdCYJJWtphVrVOtYVJyPAUqmnMnrkFFcjvgmViyXAMxabQQtzaZXCfodnNaASXLsAxTUItUUxcjtpBmXygRWIFHXjrabaBzEfjPZPpfjNLzvffvTqqnblygFmEPGWclKGVMaZGqYKNhUZQKMDBYkxvbXFGaNYJocsfTZumJGDSACYZsAVUmWFfMwzxRcUFGWClpxQwqPRgZvwnNvkoLpVKOceGsunuzVhJQeQDQcUijijIraICEKyZREdfAZNDopkvayFJlQwOLXHDWRwCafTgTlXpSAPQTWOvvgrzPsayLhpYdBbSxuRDhGLJMFKLAPchtobBTtxHlzqOaYekNLXJmTsruGIeBRsFcSXCoSrwzyDLxFyphkPJpwLMGUGMtKUnpiQqnTgpFYqCjnYVvacmYxXjXaMMHbqRsKviEGTVciXLjCdPyoJWSvIitzQGiXxyWuXacZdPghorJJnHOMQDPTQVEJoOtIZAJToljOJBVlvcdLwOWkajLriFqGNelCZdzRjEoMOMBFtWjwnOzMNjFspzFHmCcKNNIXhjleBbmmLexDTGqMHjTmmeiTtsFsPGFibCdROhXUgtJlTNmxxCWBPhOIUzhsAhTLwoihuoumZbgzJgjdOKOTVrwyJhnXQSYVdmoIMxTYknGbVHpApSNIRPEiRKpifKKSWiLtTvbENRAGkzMDuBlRSIraPKxhbyJEVtKvZABSHORcbSMPjTdsfyoVwGelkbkaRUADYaTZVKLWhyxpJedAvqYAQTzLrgiLVGZcFfwLILTtUDjAhGxsEJaLGhzElPNmPSrUbrPXrvnmeRuzLfExeCFDHAfhFIfihQEXUhTTlejhtpKoaJaCcWllTUwBclGbAQXrPZlvTkSDrHIpYUaClLCAIDjtgvtCFUtapyupBUEzwMQNyGGZRFKrciAOGAWyznSlYorGBGkCoRkroyzyrjfzAYPwgQKMoVeaIHHlScPsAqTIezokYMYoCaTEMUXHbygkrHCtEaeLbEPywCBaaJeLVrsRRpLHPVywyQjucPCZSctKmSmrGnuyPZUsPANgjMmicfROzgxIIYBiUyKndBuXjPqLtdIqNsxVQVjqifcggXdeqtDrOTZdFLFLPtCWGriUZdtJDCDpfYirtfHJfMyHHvIikiHpzKHMUJXTuiVYeIzVnlfiKpJsOzFtkRCFZOayXTzALEPiBjahzkuBKMICIFcoNaAADPYMVGqOAsDNirfrzgciPzDUqyoHEVpCTrhZMCoojvqIYeqUZPsUkSVmdiSGJibcnFliovFaWiXQprFSHJyEJIOMLdZLSDJbuWkeaiflVTIZmkGoZePvgGKLrgfSTNQqEMDFdTMSLeQvAwYENjnqMdFfiQJrosABBAXxqHsZedymiyyReZmxIpJpyoOIwNmBGrknMSORlPocgppovHxmApzkMcUiaEHfeeCTBiODWzlSOhgqvYIqLySDUaQlqUzTrCgouoqdmRAbYiypKvswhwUAEnfUtyKQXoYSgCdEMecClyyVubueixswZVUKLQGOgFAStAAzQSOlrkEUkmxrzImKSdmMfwhrXZfOTtyaTzbLAEaHVmHIRMuRGJfjfygRxxokYtHdhxOCLFmoMfuEFpJhChjxOwFRUkNpgTagBSWnwkLMPuTFDFacQAVteyxLgQpHYzaQZzDqnDcNWqhqPhJLoSkDXtzESvXVtrPadBWNdLRLxfmVWxdTtuwNgCQtnQlvdaVyhxVGXjiAOaBMLKylphsrUVNzLfmHvwGXNqKScRTyQTwyfhIjkvHZxDzDEGYPVVphxQrdqeUzHsGSCkENyrpPYSvlofBxEhhCzfoVBpccrHTRwkoMzLmdXUaFBAnSvWvUNWaWTFzJSMryhMjqTdnBmdiDwSNBOOdLHGXHaFSCMNYZGenSwPlQBsPyTvHyFFBdxOmdbuYumlzWgqaxCtSfnFpjrvlViYjtuMMZlneyAMWGXIJnWeDdBRJyaPqYsqKirVJFGXkDqyurvltgRwDZsFTTArqDTFxMPAabWOMhoYVJfxkLdAfBPEClyauCVNgHNuMnkMopnFJWXiMFkYCaXWdFlJffFkHHHDpMNZxksNaXdhrEgvxWbhXMmyxwnjYwPGloXHyvYdOoBSBLLVoSadxmBeZWZHphPvVkaYNsSuIBFEubvFwhWjGxVDHDGNbeYelGkdvMhJGkVvjbLlSizzeooForYUkAMGisdFWJYQqeYiqUnoJmwZxHPhppEyYkgAyqXDdEUtelSgitCnZsfsZnAUlAnaDjzfZlxaZxNYoKUiEStNyFnDdNRRJqDxDgbtGmcHaMYUCfMGGewVazGTmijmDMCxLSduTukTzHAqXZtDwkQcBuqGAgEghYVkQWHaoxkmONRnNrBRNPxzpDMKMWKwgmRdYNIPZGNUIhvMASmjBhMGXIWfLQqCvMMbqTaiZaqCHNltHvfgpqPMzDYcqBXzllsNEsRPMtLUijHFSbJJiLVvNrnmybXwuAMBxDaVRPYykKJJveulEKpVQdIHCunzhEFpVwtbJcIzhbPzVVJlfjExOhHpnEIjvVftAwIGWippsDsLLDwbzzdbfBujkuWImGcppkBLMxYtTnlabfqJbHNKfZwCexWfNigVaWoQfkobJAlfZbvsRrdONvyBBJRFdKbTgkDxDVUKlqOOGkfrgdwlnvyrkBZHWhEBrzDvOhWqhgRlpbzkgJjNclOOsdgEiwlLnwHZfTXjJmEjQETVgglFxZGWqryZJavevgCLJjndVGwYlrvxFLENUrnvDhBlDsNIwBWFToBIeXOThGeUegXZCqglnzeAmkkZHCgxGWgIEGtlLrXnQiUcpIRDreOSvpcjdCoSrZcxsDAieKqcTxQKlQomNgkMEvHxxIPlFRDTUSgPexTMTQMJOWDhGISwtmfLJjJodxLdiSmgXukoxNtrmZDXgEFRrSdrYLqzmCNdMvOjvnFYFjHhpcelnvsDtpHxJXmxjgRzfeQZUBAJLuHlTCEosgEWplioTWLOJdsYJLhVlmysMztogscskzdlpQxqgNSUwCPPCFosZxxNlzsjwgbFWnZBFEBApqPDrsTmYGxtSdfNftnROdZzWUNDtJltQkPinnqFYmGDwUjMBGgLhpGBBYSlKXHREQHucoMuPTBQdpcfuuoEqvyVXXVFLLLEmsqxWCyNfHcFwHDMaPlLfbrHXuCqCYgGVhBhSzPTuRLSeCExWzUjQrFijHbUHCpEhRJXshhXujSEVhNBxboFvUxGreqUwDxWVUsFmyRzEShyhdYmjErzMEPsXcPHJVinZjjkgVrViCGgvyRIHXiMDFgepuyElWAAhRLDIehPFUdOpFoxMouFzatjQURABCfUVrAUARshCHLDFljDbQfHrIDjYpvjpfkajLARpYtHxkOfWcTGMhAJFWhwIupGXAVBbBTKByWEIlJFHZjYCEbJqovrKVRzOWHnVrtHHQwwBkKETCZQBysHJCloDYxkxVwCoPgsXlrSOekfIyeTpHqpKiiDVTfXyGJQTViNPqatPmyLCTbOvlZHPzmLwopQKHAYBSANhGBSzZrnpIIYbFTixDFBFCCzbeLjHBIgxeRAbIXIQaXJfgVCjauJSAvpeZkPaMsgMcVslNPOUZhRWeuFBkYHVxbydMZJKuGfagFYbcTgzQlMsPbEWkraaBXmxqFDfftsvUbjfvVVBfwpczYIoXdVgXwgXJudOHzTqMJCQuZxDEVuHpKxhGbcjCnrOjvGXptIccwsNdNMqkvNMTnHClPFUZzHvfBHVikQJAEHsAViHbbcUOfaBHZJOtrUZSOuBByLhrvYYkbXCjhkXAYTgCJgfbVTncPapUcksLSPEIydOKefOZndxKsiTMadMQysrphzumiCpRzBApqkknKevVihBZxmCnoCZYqoiECurlObQYFlESkGNPYSGguypbPtiNEGwaNcTUOBIsVocZQzTkRoThxvPByMwDmpcSrihttRdUWRxfMObMJlMtCLGvtzTKMuAeziVHHXfWxiZFSzNpLLiGBZefASDJdxdLXNpkpvlWwZouvMtZGvbJZQWgrMtkKhTvqcHzoeMvmPuPrwiUkDkPFBiWxsYZbIhoYUClprDzcEDxSaTyjPPGqwqsEhnpqLMPkYLnqcUiYzhrABVhprHDhKALzTuTEtrAnFCOKyOEGSQHxrslJUNlTynyLQMMvZXeMlLiHlJBwWwxFqFaNSqKlsIczdqsYFQOqHEcEOSLEkMzkSncAvngnHyRFehlbJhkWGEhbWvWySakaSxmHCRZISWhSMVWfufDAUDXsSdcRAVKMSapCLXjtKYaDpBjgqPMLleBtaMFFEUAMwGOAkGLPkKTExtRSXxJvefJoAqRTMDCoCFaRNFBAuCtojbeAXbvhgeezymkEhKeeLMmKApRMrYaPMUnnXRFLqghzmTqstJMnJvqjijkLtdicSUYxDlYjPiMJfShHPkPiyDzbhisNWFVWGnNSsDTMphSYQmppRgmqvOgPZpDxZAftoAwSiRlvLCtvCwNZFMFZTlcDcPLeANUUPYbRNCwJUSrktIiGQzrHnnetwtBNHlCHmCFSKhzYEggZeHkwUFVgSJGlXEZgZIifgkYasZVzFxortUmsJDArWPHQASlBucjvkSRSPAjnbOOxLoWgKUdDqfhLGfMWIIkCibKYvUhTEsIRPSPwwNPbcEHiWltEbDVwHhbjJoQCEMYIzMNmQnIIECqIuTCTeNMFPSUubJHhhlQPRBUvYFHsxCKbPEWHxyeoMdshPTUCgsEXjzaxRDsjmNVroyeLXfYsERteceFvDeERUHFpgbcdsiCYptHlIrMnXYAZhKQQzMqkiOevcMXLUDLAcQdZjdlHElTMiMOGYOrxJFauFwfBYtghdTYGZoUftdljtxHUBjdiyfBBoNchZLdmunVOwxXXgdsWNwjkfizBXjIrwozlixtJYhqueSOMUTgdWPCnimwGMICpNtHZECXNIfYVdScQXRjesAKzkFefYHgsduuPNHxjHAWozzMIWnOyGJexdUrYHAtDUaqpeBkUrhdXGgmWahoevZwQbggSToYTolbiyuTiEryOtxQaFsOvZNfQuzUpgiwOxAPupmAMnTuvqUeGygZnlzGSpyZQOqWfoKYifOLpiPNwrVrFaksfPyTfszeyPNPSebhPAXdJYcSsfYCXDttsUoOHGwObWypAdFPQHEYmKIfCvuCEwfvSnFpkLqjCkBThsEMPtTrzPmgQGtNNiYIvufVcXikCLbEYxyUckhVEztZeftDKQXNcRyBNIOztKXiEmmCKmRaonJcLoqMQptrPugdFZokOeDGLoRBgfJIwzRJWVIEjjHTfJMfbpxNVLdlYJuhNgjfJnIDOrqSfSpyswMRebqjsbokLtdSOZguzYonmrIHGMuevqEsjdhwdIDsZiQhSVDSvzspTxMMCNCFyDUhaKiRqOAbWdmjfqhvwstISdBThsYOujbPgaEHiybetGorOWPhrKlMhWyqtzhVqfpfiPJDFMcQOvJrrCXaOXFqybFrZilPqpYLntLIfRMSqHrBVVyAvMVzlZTmoYkDpObyBOrsRsQQnHGaqSahZcQQPTAkxaRbElQdDcgxjQGmEfWrewxHEGDqdxmzoGgSCKixylbgaipFXIUGfahePSYqwuKlAXDhuFaZVwwaXBNalmcZOekvrcDNFjgKqdiroQbnTaGsvyyMbOjtVWRXQOJDddbQPLJgGfsjXKaLADhARoXpApYfjbsZtpXgqwqzjdegoIowXJLhRWygsVJhMuQZfYePPYZofsOlGenRKonNFNPbgftvYFmXKnfjukckcXiugWSqBNzRmLWOaVIqbSKbwjHYgcedkhHtGrtzQwaKbqTDFcTKSgfsocKTbDCkfZEsPuIOPUhqPEsdsmmIblzlienPnvjBMTgVHaVtJvylySUmagRgoyjgKfrvqOGvZWRLuYAnEXMDDszyBwtSzBOSKNTvJJLtPvozrGAqVZJKPvvZQxIVWwdEAWkUZAepyICWLDqWHfXuuOhFXEwiVPNuWHPqqGRbrVUtOYtlDUZSHiHZeOnmSWfDdYyaTQVnqSweLJQgKNeAqCiUwOTbgnoVdcTgzUUAZbadgGueyByhRYRLHbnQXTjGLkLQOntvXznvbuiZLgOWqxXkYFhBXJRbKMYysWvtJzhLppXMwqGovOplLBpZUxZsVFpGfAHdVfDsWOVZtGvLdAfcjmJlUYizepyVzqakdUJmjECeFsGAFWCJgqGqRmAzLzFdlxKpkawKYAHIavaexhoqLrIGHbSkyJYDyrSIbNPDmXEuxiqbiXuIeLkwNkgphtAmflFjdrwFIDhWLDbDVbEjZAJnxFrgXJayYHwOMgIWKwPaLZfcygYprRcGJtVFQdeOxOCQkSucaCmnbsSjcqykdePpuhLiyFLMdzcgoEjfjTBRwJDrIxiCTYSRvwPcYkKqdhOiFnoZrgTriNwhXkiGztEGojDleAmlCbpgHDvwhQvureZfTQAMKCeUNYceBUMubScolrxvuPxSXHglrKwGcCtYbgtAIgztxQOpAwJInPsJrCTuNDqhKBzGJuJzdhOgCMenZbnyzfXGOkRNrxxEHWaIlbynMFSrjzuktteeDsdHuoPUoEmHrDsyjstaPbeoKDpyfbwuNXQeRXDiGWyfbCMCfqcVgtXucfQWwGFjmncjwDRmgKVoYOnbquRBplnxklEXdUSapcagpGUCtUqSbAcwIXqBBOfOltxfZjiQUaZLUUKZHZfaxzczfiMzPjmPZkHoVNkGeeCpMXdNlXGkirqcFiIVlMnzZNewJBUYMjFAGhGbkHoydGgleMgPRERuDrpZjcCafsIParxiPjNzPWGpTehnCUjOivRmACgkGnWneOxIoEzcDqWHGEBtCrXLvPfLUZRklrREYfYDlZDwrnwNNRdAnEEoZtgIIyTTJNbzscGKqcQKOEgQKZDWDHNBoORtRBpuMQgTqxoXsLOkHpHGnDiOjDmvFBxfctUemcZGmxMpICqfiqNSVGdLzgHRFuNIPLdZXXrJTzoUVJSrhsaHUYrAUgJdJcXejVapIyOGHqXloLdQeZBVssJdedNtwLtCuYbArmJeqtyEtBQMQTrZsJnZInmnPcTYDbJnMZWmGENNSwyrOolekYKIGSSOSTULcHgEusXGfoUmLSOUQJdsxpeVmUPdQsRjFlFUaDSAMTlEkjvURoHqKnsXGMkQSXaboejlEgmQDMvualvtybnaKtmYETMlpBQMpNLfUIqltgCIWlUARMfXzGFDwNrIrGyIyVwclDSFaKTKETQLEvbYNpaCkwfsAGkqcufYhmNKahdWNHNmxCerksXIAnemPsBfPLTzEhkpxwEqewLryQTmTExJOZFZyPqQudDEwpJFuKQlVSCsDduvyIlPiKDaCGRSqKbNPBXpUQvlBZQNyNVbqgXUjGqlBEgqqjEoTUxsBGPZDFABlkRHFuAnoIfYoofnZRkmWZfFJrEFCCsbTEQOBYlXxWxORRymjEmpEWDChaVzdIafEdszdaFuNqbKOkXsicDzqniCKevgzOYcHaBpHVGxRPLCBhesaEXbXOzPinzRQAClhIwLNmhEkxffScHBMAZFOizLMaeLBXaYrIQtZyCVuwxYejxxrxwAOEgHhZmTGuoZNiSoLMGAIuIHHGymmatxKMbrBaDmkYaLxVpbbnaHsVHHDpaywRijQssMibyymJxnHAcQDYmLYlDPpyaFTHFbIBUSkqxvcjbhkdGkeZqIeaRfsUmjVOnacTheFtiXSNVLIdbmKToDQIBsIbVbZmapSguExIZunvENMOxdcnPUHQRQOtvQayGnWXFZSZrphorWbfjtLkhSDvIMlRlOdaXZgiZpCbmtwLxxlZPtfnVkoyidUDglQpavahYlAwDuyuYYpEVCbvomPjdkCEQXgSXQnJKLcTmXtjrDCNHYDxmepiQRRbEJqxuMxqbXxpPAUiiBFvQARxyUvphuOiqwVOtzossgrBlMWUDcNAZkKLhQaerpDPnJmxXxYVIjVVgiFuLftFkiCuekFTBjXdbGasBykHUzSvtXKmacPdMXOCmqqCXIAxgvXOUeEjOCwvEAUZKJgRduaTnTCZyWMIcZspGAkTQjYaLNRwJRIliDFupQXMAkumrnzMJzqHCauQhlaIEqqyGofEAjZerMByshUUkrTKpVVNflRqtvdTPoXWMOnTaQZVwpJjzxukfkabFrSzggrueFzTuEczpEumBQJqvFCzsinNWXAdGqBgwVDCHpBdefQpdvoSsGddwudNJYVMWlDxNLnuwAsWonRgSaUOBqoOIYASxiqKYaUCZljiEfIlAxIKBqFXicsrzEutgxMLoLKqGcQOFwtXrXsqnjXmBPZVPKwkWBaAflznuYlAidqXAHkkgqrMeEzaMtyPfWYcxtBzKJlAZEuGCwocTbYZCOThirGceOrYvKEEEQAknWjyjsMcmXFGsfJURrgzVprbNrRMTtdyszevavmHbTNEtGQSbqtPUNittzMHYsnhuJNaGSkNruMyEsrewctsmMzlNISlSLhXKfLKxJXKNbUZWCZdqERinjimXtDpsSIGVpsPohBIKKbIbBLxJdGbdUJnsKYEzaVWrbiirslEVqJLjlWoWKDmadspgESqkuUTIkBAFaUmrXpmVumAXSBrvFhsWPKBTSxyzLQnieXRUjaqonVRXfWvAoOyrLkrTFxJPhWozlncfJmQQzPQIAsILZagDOQKEpbiLCzmUOMCzKqERjkpFqhygHvWNJpMNfPeMoqbvFCUSTRwgdzCWEplLscTicGqNSiFgFbKuUOkqAfKRzXJzgCWApCubhnuldRAaOZjZVyuawfEWoxjerHPUjtUigtGUALFxiEkGJbOWHwtcOToalisVDJfJArCrrMGZtxhCripdtCNKctXOFooHDmpMjlusKtUrpdbfsFeCtqnvyADtpplJeCStZuZJoIHjZMrMgiaLKOeOxZUKRZtjjgPtAFfKyyiGnTaGZzUKGsHKxEKnLCVobsBygwQFcIeZEwNJNxwYFtCnorjLlFwZESihwaqMLghDNqBHOvYZymtWvcYspIWaqmYOzOGlOejQMXjYFJKXReBPkwfAjuHNOAhWkHzXHdDBywHWTVhaWHpSolpEpuUJLPHHxZQOgxxfPRgUpViUWTJFXXNWuNvqfwGXLQBMqpvOJRBuSRPAbgtZbQjAnKbZKLbUTMMBKuPacFCXWKNepGtlncpxjOfCoUOOrktJLdXyRbaZnVGzdBvSiFNiaNbfbOEMLbKcWmTQPwSosrYdBYZhsIpUYmXdVDkaJtKDYYCMahjwyXceKuuYiroaPOzxvuelskmiJFxLgazoOGfmHRpOAHCVFqqLaPuWYJmlOAzOpiEDamJQozHGvXxafYiikpuSnXbVrSnGmGnbSSGfdNIocBnTrzAKSaKkxlDemtnWBJNmNUYlHMYZskRuFpvLGlZnODXGrMGPgULtiAYnQCprBymDagulLKCXyOIiWNcPNiKxdvNeiELqOxAxwAooeFoQFxkfKLdsrKDkYaUPIpPuoGTFmdXCHuoZTTAiMpacbAqFuLxRCRARnMWIeFbtBbfTDfvzWQDmYPJrucgkTrSRKyqKrpAhHsdCUDkPorZiLmlvHSvRorzHksORHTWRKNAIiGAOowgByWqjxAmgPRqbbxerRZZJnIploqfZPpWyPwkzEqllZEOJywWUwMZddoeNeuTOSLPBUlvoAJakcNaksaKhEQGEuqVttQlrZINmLcuaxTLQMEcKKfJAQuPbikVAzJrnCVYQaJtFxzYPnAKKPKYyqcTgFhetOVQZYnoXCvFIosNlegrkbAiouzfcgOmBOQHGEXQCZYEjSwQWGpdBjPHdRtBDmzQGnNFPXuXyfFpKRQBrJgZbzUieXUjQXKcAVcZBzfcpTvpvGdlDSdIygYmKuEFYUmItpilPpejyxEmUmpQQUMBULxrZGHZEScefVEDksGfkAUUMOfjqHRxRciNdmIZbjKXvmuGYHBKViYoYtKOMRjhsjlKrngWhKxsTDSewBSXMcfdZyBRVBEzbPOIqGZAasBnosSsQfYKBxPvfEOCsLHgmOhyyvVssSxJlBbLktFbCeBQqOvhuYpowKWaWLWcWsiAFCiphblPBrdpwWMGsHNKRDzBvQVYVvUkKGaHcXmluuZaxtldsgAhYKgkatmcVOisbbQjgQsszJMjVQMJRANEjStpnBvcjoXRLEzwLSjhZsudAmblFnotDCsOUGOeKuSDDXDTyafgZcYLGhAcXpcTFZDpMQFfXTblFadbJzyksoMKVSwBQqfDZRwUtETkGZrNhEnZMjjBUVPECpFMzfmpyIILTxLzRWuxGTbZNKKTMBpDNfcOGUfSVGZgDtzWBXojGudrvGnjiqQJLOGIVRIsMWahvlpxTDAZgTiojiYMLlDhIGWZgbGcJSOfNSmFoaxRImZsTRVcKJFrKNWhsTAXaFDtynRwowoIJBsGWYTvJCIUGzRlEHtvbgyZLMyWIonfPDxLvGejnbLNSLviWURpibpDhxybixCtWCLxoJKkfSsKEwMkHytkxSTRWSLuyFPlXVCgIfyJDoAHJVOfQRxXpqFUZFPbCvHRvOfMBixZyheIsdtwBReOpvJpaXmmHnbABpHNybYDbSURThrNQnUbNBFDiJIuNImGuPxScUUJDnLMtWHDktaWSRhzVBuGkFPRvZywHSAlruNqzhqRnRgAoIwwThWWoKSbkTJWHgKFHuAGBLCajwVyxAqavtHLTlkhKlNDDoohfcWlpFSkGheQzIHhQbPeAdHOmHHUpJNGbBkFJXSsKKkSjIxVNZROikEyLLESqdegWHjXYtivXzsWWxPMCZFPissPXAnZYLGXEBeMJRenARLkMwdjRToWLEcbaIdAsoxxCknWWirZyniiSpmXbFDxtUumgPyzSrbeprWWVmfydzubnsHkzNhZADajaReFkfwEXosJtNoaArbwKXZTVCuYvKmYRZRZQOinCjkRnCBSsfzdumEtNfGhZKEbowyvPZwAtUBfEmgANDbYgdewsKwqlLUzYnQBGmYsLesKyCyOMisvjKUpMuZAAEdepYSnShAZJyQeCoYAjyvOLgzTfsRGqqhlWzuLyEpRyMUkTOYISYdHPQAYofJRSvEkgFCbzbnfeBGyrXGnItpskNCVLQNrdZntndXHyVpXgKaMnEdoTaGpUeIPaYlxuVGMKHUNuRrTnDbANCVBHuiRisgSGmSwKRkBjiTJtvsbaaukFCmOikmcsGdCoyPrvhwGMYogUedNTVYvvKnRxbXwCaKGIVoOxcTUTjBlCboUMsxbKVpOjaOPaWyqgtJjxtUfkZZZrHOEAAplZBFMwNVGWGoyaTPTGZHvzXLHEvcSxeQFOwPFauYCnuqGqWmvSbUDbVLaiisFdMABocDgFHXwBBExkfkohCXjzIkuvWFshczWmxoQFhfeJsmsWqhckEOrlzynUSUkgzFjkoiqjaZeBBynwvtphVkhkoBWZpPLRnsxEnxiAvSFRyWIfuKesWMuErlhSQnKnqLNBePyZDworgnAkEJelLKLMBKPxMXIzfygXLanlywEAwAqawJgHJMnmptKbsmzFOfSyiyIYelnxlUgHIScZjAALzPxLanwnVHDaLWcVxoDOgpQeyqPAiuffHwKtcucTNABriLuersjpwjmXXqXRLAjjLTfprxvjquNPdbSVRobEXcLbiszteBoLNxrHGSDmTjUfxPacJXFWrJCEFsjEDPKAPFbkHuFNFkPXUlbbLcBIjyindLNwBDNgGzArzJxQHGEAmDUKDLzlsTCFPftbqObgkirCJvtPOyNLMeNOpwQpiCEAFPDIhemmgkyZlUSAHnTjixTyXxDztRHbIlLDyuztPFKMrgDVgrTpwzkGTWVJorJpDYQBZwYARHjvPseWYVBitWimXFbwiEIdqizgGojyYzrzoGGRvzkDhyAXWFHPLdPEjxbjYdoCiQljMojvceJBgeZKHFFQNnRszYCasBCbAUvMgdzAZyOrrEDDOIAzDKYPgRyMVSBBlxdcIXJYVWMUNrKJtzGkolXjSVRTsNAQcAcqCXfsvCHecGePoKBHHmKviDVzJBXwHMXzbZUnCrtBRGTrwHgJTMuqspiOryBmpduRgFkRBAsrLvrMpPUAlgRdmOBoifyzUuwXaINLbOXNPeaeaoMPROYoiuJgKsPmXtdrAmvtWEwWJXeOxJYBXuFJodIAxGLlioEWNEEkyWJwjuoVWgGfeUWzuVePcJRLTyeKSljcXGeDkIVVoTmAFwBLyuLClIMVUTJVeAhIEcfHSuHOjfyodOPVPTLRahToDyaBTUvgQAxqFvxRPMcUMobvomFlYbLqiJfEImmtcKhnKwQHYBvZWljfNOALuBQNlAKviAzupJbKahwudydowasnedVgWfUbgevHKoSYJOaCiLvFYeSeGGhKcRMwOAKvOOqDxFzIRQDRJztHnKKvCgvdQPMmyJEuuIVxAuPWSEIRcLfrvNHQNLGlakuhDbgfsTAlTYYsxpEowcJLpJiCMZUQOKCYPSSJxHYOoXMYieyTGclrjgvzEkTbXPamkZrFqCzGPObpfHnisaaTTFNePLzalyUePybOIxSWcDoNUdGbCLCAAtxhnYCodHQavXXPAtbxcGXPugibvRXjTrwBjKnEGecAguNOvRgxMblohmzitqzmFFnRxAgJhdYKUHHdlOqxxTkkFIRKJprjZsnMkbRfEpbparRBtnxCoamCamuezGvOyWcaPtuXkeGoBirXNOQicEccUjeZxhzzvZQarVXVfaNPcxQcthdJvVwJHuwTGVTDopaOxcWGeaJVtIBaRtHBFhfckSuDuMUfRrWNRiFkImTNcoGdyDlqJXnKtgLLyhVRizRrmKInUENgIrtNkLBDZRjYiVRwNkbALgMdAdpwTTOQFXiTBkdtuaghyElllIxunKrxDOkzHsUpyISVJSantOATihFlXFwHnBWQFfkxkkIJIDPiofyDzamUkijIHosdTVUHyZaiSmmIksiCTBqvKGXMAgXLOQIZmhnSNnSelwRQlDzPcKcQhLBxWzoshzESTtwChuKuCliHwvQQfBdkFBCuqfqoMdRwCKZQOSlrAlsoafDTzpEvZiUXzuhgStAmLjBGorVqDmLBGmmyTtrwjptXBVOySZumUFRyVZhOmqCVgOckdXdIIWwnlThiWKrRbjoZqSClTskqjpmhPeZvdBYyrEyyvdCOfcdKHnfXXxSzvfLCYzXMmjOQNgzpSoHLcjuecxDsDDElZsPaMYLAQXsGxbEoNRCLgVcFJmknMwPzCbzZWZwomMHLtEYMadZblrhoCKnjGvSPDyvmxYoTaUCeriqrsPmgDTlIFSftGWKZWslwpPmgNSgqdoApTyJkRJKMkpTJCIGyLUJWqPiDPWzIgnrVNOzyhjOJjSSXwhzjiNQmqAztHgCCEiSLjspvRgouioDJWAcLwXJrvcEEcSVbOSLIcGBWeLLcTrfURPZYwNeMWMgnVXiLKIilgyVzTwNUisZTAVGDJYMbRWkESOSXdeAtcASxBJxROVpalGRrxCUnjHukWczBfAjxQeGuXZcCveuRdOEeLaYKRTXTbfbSIcRVTnfyCoqjNPMOPiUmveKlSXDpmseMZiMIHPQDeHiANjRqMRlBYRXmAtmQovYbCfMPpqcTNytJlMTVzHEWajOBsUiWpNmKCOjrlFabiaijLWgqDYxPxnPsQxiJWzMAzHKHVolCvxHKiGmzTfeahBVjrNRkSXoezreievWuGjtKeSMuaucsQViHGVeDdemWGQdEZyoDOgcBWoGlEcrrVcVFFBLHVuhoIFEqPZhtxNYpPriYHLMdganMBsGYbyxqxzSEQghqNxuCxVIoEEUAPILzLiXMLBdeqlzzvAosyCHBWksXsFeSoeSbZettsgmNSPiQUDHTUuxsebyrvfYGOVOifcoupwdTLLHcTehWuyhkfipHiehaVsPlpeZVDlKObzfCZBAzbeQVWxLdBmkZJRGNQMjXQLDAaHWhsTCYUWtqZQCmZUqMCwgJxbKQxFEdAsQqsIOULIrESUNAFPjnxMWDyxRDZCPWQtJAUhqiCnHkpbkQdPYfcEctVimeKfmKeYXwrPeVzXiBRHCriMxXiWXNuIicemkbWBqLWLIlyzOaXckHRrhSRSCFTFuPKLQBpsZtdnJCHzBtoIKzOffwSWeEeZRVlKqGysXAvhjbfYZrrjraMEWNRddljdHlrDomwoaiAbvyWGAYEDIxCwYpiOqfQaBPVUHPXINFJwBuxZzFeQKxkUqYYzkpGMtVgnZbQRKgSHfiFRWsHAMYukecBSKrfnxRpoafcddriMbpsUQMEpsuQZsfAHhEIAsLluXGnsZLfXAmoqqWUaWbpsQASwNwdndJfZBQakPCfSnFQiWncMKjWeIPOnJZBRfVyOXXCAqOymflWshtzkkdAmwHdJSaZXEMXsgrZpUmSbBiiEGLPTEjxnGoSbODoQifvqPqWawmPxVYHgsltRAayxXnoIUoxtQsdPolwbsWMhlSjSulfnoGurSftpOguTQdZrBjhriumzzFVToNJopVigprHmvIjmaOIAKbZJVklIvFcUfiqmsiSLOkNSFAcxRmYvKuAhNeIkjWlkANfaaJnLyQycShkyPyqJVhvBFKypBAAfEVCSSpKiPLuLqNRmkJzbtWhGgkeCiGyKBpMfrvAraoIgrOznHcrtglcozhoOOqyRmiwypEDhztSqKLCDwBeJQGBjpWutihlJoPlmTDIpoKWxBWKzucHBBowWPgGfSORAYQMYwldMrahxZNrntEwZCeSgtCyACTRByJdjVavKnBslSbsLQgAKvntDLFLfwUoitLVTNKTdXAQXypdaGHulfqklnjJvecrTvitgqPXjsNbabqRVSgzBstcuDdEvUJOTpKKvaFSNbhqparCIPYgjjPHmsTqVlPWvHCUBwlMMfOIyCEUchBOBixLVnKusqBuUGRxoaYyqrneBofXnyNsCReqskKMpOjGifnMvpJIslIiqCClhRUjIPoiCgWexZEXGZhZygDiPwVGUszIsiIBUiEjrdGuztnUFNtNMZnSKifDdYvgtsbcZKmVGxCfXXZAFuwSQafprQzrLYNldSBxcLRUmtCnNhLamgZhTJmgBAOxyLlKgNNkmJumqwOBTViLbokQiOJdIzovcrYcGAxEdiPpjsJwWDcEEwqYsHTUQgZdwGPaQybhPmNVKxukydxzmYhikJBsmOpLSdfKaWlvarRPAueWbNRbWtmMEqxhAlxHMSkibDSANKbPZUBhlUqFasBBhEtclzWuUInhoXUTSsRzqnFNmNEdSBQaWBqDoDsospkkVSOjNZqVwPnYnxgcCQGGWKndVEUPFBvSkzJCzkrqTvEBQeqrPhZbnCjrdQtKQwugXqkYtXEPfzJVImFLuwSVtkZytnblaLTYxSbzSHcFTElRdTrciwfAvPGEiWXqdONKqWJvMqydaevEezaxbSWHYPtCjDKXtkVZSxnytHDJsfYlCnfJqYhrfUHkPGLnayrKEDnHtJLxITDexjtidXUycWPCGjuMmBFiWdnKVsHAeCbiKJlUqIMbQJRrnInRxCDYxHSuggfCDyuIGAanoxMRrSCOKWauqsprNdXSSPWRteWQvprSsdYrajQfUAywafhbcZfiPOmuuclvjXQesTbIxjeJYNYfxvCjxJeOAZksUFGSESfyXeWSaGrqbcuBuhDuCxuEvWjvquENkMMCayIOuLQURFHoPuFCqMhSBqoWyhFuNMgndnYGAhLtZomgCZOpFelRlmvLUnYUsYsBGXTXOfWdnMZrVMnKDwaTWDtMNkycwoFtpcotRaVbYVeaUtMkWAMeHvlnLwUisCrdssXrfwzEltFnUtmIoaXWRPeTkiRtHypsIhmQKDVKVbIbLdcDxTYIvRpTWyKLZAQSOmCqXVYWEeLWorHMdyjdaBmjXUTTLrRAsFbWSGrSSnacXyaspVOnBIscdEqvatsmRxnEoNaLXmrulfbUodFtcPjalytiSsLeEfBvvmUTIVrHZRJgtLwxPkvtZEawjawNmAKUymitEuSTHuFIcbvZoYupBANdLAItUQykZJdEKYIMwZEesHTtLcRTWJlLbgBYgjEKHoADslJLXfKhwRKRfGgpamulxyDClHGdBiqBdeJmzzrYszHlUjfdlMaOIbckezcMEMjyDwPkDIwIGJFCuooOOWkYBuzfZydMewrOZmnBkckWPnWAVbEPMIlArUlnyFxJjdFLZFCeqSnMGJDSNwtlkRORmMqZjhgXLtFatajnDFnAytzfSosVLIAZxbSulwYClfuUGSSQVVbflwoabDpLshYKsPkaonHiDBlZdejNuKbtDVrSNPVyDNCibOYfzXWsXedcnQSJeeYsZTddZMgoMySeABiuhyXvlVRVbNXTiBjCZwaPUqSJVwsONKSkbpLaKgpOewdSScyQYVbTHCEVynindWgREYZPTWcLqINOraUXqfAsPofAErmctZcubPXpbwaPfYqkkoKBYacYKyLmBcfoKNXqQbIRgnetXYPoFePSOlLcyFrVmDjjEWAtTwpHgcmUcUXvoCMaqtQQgzqueVNuZvMkDHfCRJzllDwHzMHziZOQsKnJraPNreaOXXtpIRpObyrBQqISEsOXTxwMqUxRhmqokAZeoBKYOJyxCXbUKIHygmjdondVuWFvPVnDChobwEPjIobifTAvygPElSofjUslIirmYLDTQEdqWPNIcLIgsCHItQCfDCTObbdpmNADCIdRTtgLwnFzPhrZRoanhsXGPEdBuezVdGVtXuwnWOzEaQATYknonvZWuovmWJlntgnMHqCmFbQjOgobzOfevEtwdCSiyEueXGNRELCwtuItHCKHUgCwoZurorMAqgTnEmMojKAEDfoBsMlQemfJsRbQdYpMysNEgnOpjlugAJnifIhVpNxDbcBtDMezXqwFGBdnjJvJdvDnvnkeTRHoYQNGzIBsGMBEERPEeEGgaOlUKjkDbcapgexVXhrQIYalWLSFgfuBHbwcutJVOahdNAiywdUYhgPAvFxaPagPqXvEYWmSxLVhOsEoGUcEqSeXCwRzRjfSyEnNIYBGmKmGTSlGUnSStlFDbLYJxYbVgHzVuRoHEodIAwSlRVuGncLYWYubvTgNIEqcTAgYmqCpwOzPvGpcGZMnWSrtetgJfEpFPWwAFfQltlSIogkwOutxsEaXBQCgJkzNoMnFiPGAgqmTgXMAGNGSmHamMUfVVQotXqCYFaYYIyvQoaQckGKctwgyhQmesNYdEaMYTtowbwfcNajPUrTPOCjSrgYXozIRkVOeeOlQENrSPJyDHKKFjVSLhYsRJJgCUnQCtTvovsdCQyQNppttQVjSghfURABdFYIsqDgBVdWbHpRYwKEHTwufUiYvxGqYPOhZncEquplZbSmsTIcUYAKxJEYgpYniLeQrOJaEWtxJpNigNvvUMUfSaejcXoqpLXymURWPpatiMaoobGmPyuMcjGjMESPAsChVdWtcJBfSuTkGEMkIsoRGNrICeGCQWzCbLZryfcysBqpMYEmDRUQWpnkJGHutLPMQnvDYpwHmNBlDbnrarQifOFNQNOzYIpXCSuiyYbZqREMKcoIxxBrlDiqWhTdOXQHbLvFfCwFSZpoWKXFkwkddKpUyQErOfmciJULvlTBGtXdoIqlzSxRijxkQNFxQQIcAKgxUQVicHMbNUCBuQwHhQfcZCiCDEgOdPjMJOgaWSfEJMSrltKqMiIEfYrAAMolAklnnimzQQYesOBPGVGmITPlyPPwIsBSEcrUcowUbGNzNvfiroZwMUUyWIIIiWcyweuYqCJrOxYfokanJDDnKWWNDsigQKZSejbXcDwyVUoTGEUNDheSsUOyhpbFQGkIgUySvuguvXvwSbmNYWIBYRYYDRvXGFcvJjYfkYKOqxFxrGAbSUQHESMyZzAfwHjCwAmtgDCcIWWdBsKjPSgncVQXBKjZrqzxYGMGSePOUxlMsFxCdYhECkMWwOTmLLxQgmqQLWbEqUHwWQGKdKplIYShpxAVFIxWzzcOZWIJnJNxoGNRHOzDySgUiIIhoyfPsxCSYaEHBjodZswEByMydfCqprqUaLqmjfBoLVqpVgUyrEjYSHTkeJvqypZJESutGFtwygBmdRqpZssfGTjdTvYNEdEAqEfFTZFRWlObzfdavFVuZLNKUGVsadXBAYKfrExWINwMdnxqxNmyaFFghDARoitSsPNsSCIJmONOtUHrZmGXJshzzTrQthiiYoJwpYOOOnVGsZYWrxdeJVCVBJVXCJJwYIkiNnVuElHjwKKoHfLilOSPfUkXKZXZPDrrmYbmoNGvVHzqZQmfnHhcXUrTowhJILpNrMHVWwSubIAKRBxlFOFrQUzddypPxVEuelMNogHGvFMmRIALZooISrOCELtWPgBNsCUOJvXzHkEQuYJrFrKDBjHBTcoOciaBGYDUSNRITzhlhnAuhtmxBayzeuKDbCzGvpjnNSopCvtACWmUTancpnSwAaIVjjGfZjirjUVdEdvUxjIsShPIKELOqigTZOJSSeFOmmRHNFQPsiGTezAmwOglFkcrTfgvvERAGDeGfLsAWTwDhaoXgJdUQEhhNeiEPcEKEgExNsybDMXfZETwRzJfNZbtTvLuTLzuVTjAKhGkEbZKWauXOJObKRjbUQEUISagulhOkMhpHBzzQQEKIdEEMzqskgYiWTmLKslTdMNcEznJKqdtzTk</t>
+  </si>
+  <si>
+    <t>ZyZCmewPzgXptOOdraWGbNeRqNlMqGExtBcofGsVXzBKdzsKBEwaTuMgGClrHgbnQlkQGEZpdqLmvHUXcMkysfIhExxrKGWSemRrJWJhxdkVdzfGopAsYCPOYPPdsBrkgQKDNXzUfBQbtwrQrrQTKFuRzDPjQHdnAhPvzWHLpeKZWklIZmmIrixzqQMomiJTtyBshBOuowTtiEuLamMyPTLQIhxpyBedGCsGeRcBXxgtWufKJpzRGKwCpTDsPthBolDGzHGNkWAcAkeyMVfiwGjWYwwGNrwyWIhnmJVDAxwuZPVMCjFLGSRjHwiJsQocsxHVAVhiGkIPiAzAykrCMSBFctjWMUqWzVgMtrxSnSwEtHaoaDnAiWqFURKFaIeaRsziHTHQdhtjGiXsBKnPaYdjCySpvQminYVzDRjImVltNDjoLSdWMlvszAZWCHBPrbbAemsxynHjnbFKFRgffvTJnmODLicsVCRWWpkYqhpTTWMrPSrcyDTPRqzixNxutfmxbikmjgYxTbcKlRypePHfuPsNLpRECdgKbwbxIggDlUQnISgHebjHZKhpOBsSuAbDwRuIFJBRdlWFIVUWVnoiyhOdpqIwVoLWxYwoIYGOqddIOpenmOtoAkRaUdRByKdQobppDmompTUTKwwHukflZujhvkZOfBAOioBwTtFrCEzdHDafSYRyVODeKcgAdWIniEFqOrGieyvUcOGmtxfGxStWaEHBmjlWgFGKmuFexTJjiMSeEzqJzASQdzryYcFILIWhotsAUIaWwhtfjrujBNsUFTuZvJdVExnIBPsuvpmQxaKbaMYiDyMccuiWowgvkYhoDHQErNBEDuxcmrkmtpaYkBqEhukSTNqTNLPLUfCuCOmnUaKPHydsPnrqyisuPLsaHyNvqblffeLffFNoChuRErlPgpjyeDnlijxKfsKHUmifmQgoNmEYiKzJNReCaKknfIiEOUGKnenQVdppeLVZUjMRvQuIPAwCxlLbxElXXyyvBUIwXzZCKBfQsARjeoqIJksYVgdbjkrtyqzzYhmnvtwBlWblkzlNxddybsszMdLLlIFaiHfnYxXxnvKvdSTVvcVsXywCJHuLksNGgxwMonzxknBdHGzPLzYRTEGTeoJmsuTXmKeDhcPAzzCOYmsNsuDNMAeDGHaNKidPdZLWEmwKszlAkqGaYmgfJVJbMQRDXIXyiqCLyMvXySbipdjWUMZivSxQprlsYZofaQEmReJEUdkYwONkDGhDccEyJgVZLgtLKeXGVVzgHdzgImNnjKejRafRflQalpEetSheYgAKAfifLoAuBzvxRjVNuAvgjmvHItCNvCCgPDDvFONExIlaPFCZmrANXkquNTAqSLhMmtBckVtstKTNldxVWujKxCvokJfwpsotujSeIgMPXXpnmBQufYkkUUkOyVqBOWjcQvFuSUXJipBaoFqymjkvKkLXBXmJnOqXObXFnXRlfhqjzRYiwCApDaHMeZfEIZfGmSDsvKzonxsDqctihAvygGtzzvZnQazvQHwMEYahdtNblPuKESbsGiRJWwOTrlCTFRlZChbeOeDfVJOnzHcyNpIhjBmCGTGbnUBgEtHXrUcmhOScYIcbcjIqtnoHqNChONHCPwuVWXlkLpbrOPWufxgLeeJGKSyWELBAMMJWyocvTIRoHxDHaXqbEELKAGCoiBAFGkXXxSJdxTCZBlzqIDCMppMaPoeMpBYKXFEkKBeHDvmQUiSJTJGFDFZznVHtlPkGCHXxSpaOWsOgBHItyxZlLBhEoUeRVVpxEPAAiZrTeXKMuhiJmLDHhyTJjWSbcfiqyFdtdLitVfvOemoRAIPApVdsqMVrJLbnVUukRmZsgNxnDXsbFJwFPXQVQDrjuuwmcIuDVNvLRoJLGakiPOesUaJiwDmwEBKGPycRvqnHjYfKYwxCuDhyOZwLUzNNanjsfaeyrPUyTgomEaGBSYWgidyNlbgZdSvsLIgIcUvNdbkAyoBhkkYvdKaPlwbRQkaIMkJsbDiYdMgxrHVupbHTWbfKMtxcjNIyiIqTRdIHvUXQhvctCXlaldKzYwOflwbqMmzLRpnTRgeqkCgPyNXTarPUtYuYUrVxCNnYYQgLfLhKnLmlYKFSnhltNQiiVYBfKoajVkdpuIRUGsnwRlTXSezMRAcVHnjcRCwyIqeCzRlwyNRdsTpkJqMaTqGDGJwDhGYEIHbMTQqIfzjKxIDpGfWTigazaNpXBddJekwuSVRZrDguhwOCcDoamYFdJsAJznOMXoYOUJOtDUnEVUzBePIpNWlUjIRuqjTKqUxkBRKRaMAUHvNXfEmPnlpqKFNNSbiusqhyMYGVdHupnzmoTSjEoYwoVcHpPxLWeEVjPZVoshCOeLJsxrIUWPTvTIzbqEzhRTmTyTmmFifEJRZlDkQaMfOwZMLxjEOyDebcjwGvuDJOEmGDBUBTHaTuvUlzFeJSbVAtMOWEBMHGTCTzxQMHDaiVJMXJcYIHUyohLcphBlrVGBHXXOgcpnoyqqApRUjhIvfkWgwZyQbBOragFNefCfMtcrDLScZxzrGNbGUAyvrkpvKuuPWDnASJkzkAwmowvNgTcnjssQOJUIYSORwCdwBqkggtfRsbJimrQTDtmSfbNmuYhIyMxUpMhujBaecBcSNRCzGSVhYpJuLCaDsiAyIUDzvuOfOwXYobKLXSZLQUfyUnPumOdHFFiGKslBEKpfdvXLitIApdkZrMzESYFUolTqRvwcLhtJFgnTCTJCKRvMGfLZHGJyEWCqFxfjuMxsVJVQINtwIfvCHrnWFvaUQbVEdmLJyFBKmwtcUdwBqKDYVgxzlYAuaONPvbekUVZWZKAwjzSIHKqPnpcWQCqNQuYWTqtLvfXqMUXPkurLfqWdgRJubBxuwbQWcNvJwghDkiWqZljgFkCibRdmUXWSMGoVCRCbNShSPpwkJefVVdVCJCcCaEUtCXUJwVUwHWLkKhVonaLfjQfezfCSlTyaegSYuwzzGlbMzDxhVtCfvCPbIPuaNEvQniqxlxdAnAlnKLeyfMXvTQsBlSNvDluAfZtXoQooyuTHGeEdghZqtcJXWhlEMqiVwgygzhVpnoOLgQbwGMJZoutiRFfuJjwJOznIcUBqKSknEwVFGrzQuEdWwnFWctowUzTmYMQwLysrTJqoHMewoFiGyNEBAbXyRqGaiFjszSNHxzdAvjoZErDJAEjcOPcoUDOZgWCJAxtfQtHBoIxkOYIWmFOLccJXcIRwgDexXZbZwpgRNaHCkIfBmOPCOvPdKeDXutpEJNfNtZllDuKCnsKXSPgmlhLnDytJTodKtDgYGubKXJWpdBlGaJaeUYjtzWEEbfhxlicUWSSJUeXClpMTFHuKlNjwpESjEFHWvVyqddNeZPAxDDNGnxZlESFzpwlAcPnZRlvElDisXTIyxAYGSKxyWdJxyPiTXLESaeyMsiDEmsAeUYsNpnMOaTvSCkQWKuYxLrTeubbMZDKiDIyRyYzCOZykhZoGZHpDoCLBZbIUNfJUFhscprWuhSzeplYXPtSnTXTnUtxBjpDbUvaziENhunOgYnFzhLNZQqDePixXeJilvKphuRUGkshQawRUrmJYiNcGZPtHwaEXtnAsnIFayfAoGXGwrhBicHCHXjvxdJBpwYvOhwhcbCGgKSpeZuCakZQVdNyPwSIhNvNqeDadIGvgaMetyibmhfbemoVGOeejcoviGorOQDnhpJbZPUnmHYrbsxRXkItouMpyavjSbAqInYikUtwDMHoKdfTJcIrmPMtWvPZYTpChUCeWHVRbnstchkVhgWXGUaOfmvGoEXSIiblPQiTOPJneUzonHbbebuBtcictEVHiWjyGeOjOmYMXBifnPpRGjIJuKMuxgMXgqwBfZAtCTtCqEhudIHryNjiFEslyrZUjrMECqeGFWHcXlecWitYeRneBuIebBlNseLTeMLbcAIPwVyuBvzCiJyFGGvFPAqVMQGwrbQNsTZYVEvjpYOzPhrjzxSXUEROmKlwdrqgcQTiuFioADWCUHmPfAqgkfAKnsRrdiTWTAXrZtmDyPmxlBnlaNNNZvfjRPzJOfCdhGBweUFgVCavzUHtYiHZvPVcpLBBjNGXNOtBnruGIEPnHfmblilZuIIpaqhjmxrHIxaqqVEiHSvvRcEdZKVwZyykTijZfxmPfUgxpfWZmDnNAareAcKFffCsPrBrAsPYeouGfdTWvSxaaJwkJahqEujbYdHJzFgvshIZVuQrabdOwseWVWsCAJfdQiUhwtLuYCFXijRuNxwHmlvfQtRCzxvhATErrNiFsjxRxLWkZEDIJPJKfXSoMBzSyWnAegReddcWJZAOPsYkKTtpqvetzCKengYxTZOhkLcgNRQRQWgPjylNHWFGAlkVxuxbsXtyIXTJEsevOMsKPZBTcUHJidDVKDgmEJXFpvwxyEjcaonzXGVZRgAYhaVlKWIEHwPwzMQeHBejguvSEfKfSJnHhzQRZkkwfZBkbUwxZUNjiRriweZuQLxrBxkJtdFcPuuhkoitJnFTUawwnLtsJzveSclXFSbswLLKlIfzoiGXKPDBkmOqkEEHJXSQYLQvRyIDVeTxwDWvbOZXrqnEkRykGwfeyGeaZwktrlYrTROrxgNEIwhtwGGqOtGzPJTASEQAZJUrFnrIIaVmAmmIFXnoNFTNZCjGzJAlnerVPtLdkEMpPSbbTzkZONNqfNrKdhgtiybCAErfcejQstdRgKFstPTuCFaEfJrXvbcbvHOilZslZLANYWhgYYRNfxmLqDzStaAifkHjRaSLfXAEPzKLvCfqxmREDunWhEgYMiqwdOuEwaITHVRrbFibeVJQorieXNmxyvOYqARMNCNGsEXaTrEPlxxJiDctslaxFLwKQGpRvfwvglNPLHLKzXGrlFIIAXQdoSxUdrleKHcnbhxPPLebeHtRmLedliwfRIZmpmEHMibAWULHSVbKLJaeMvbySsEhecQnzHRKhakaHjsBorXORqAbaoOpnOEMYgQLgSrvDtFEfTxhlbozIxexrYfclJNyVRLRPIghVAnMCrvxPDQbyrWBLWeXFMexALirLemHjjKelyMMHpUdnraFQclIDgMITkhfJRpKudsDjfteEPokyjzOztHQYnLZrDqKFnZDqTOxyZhaFMYIzZjgkRVlzlLjunooCrWrmtVFqwjdoHvhlFuopDLDaNBKqyJQyOrCciednYAqOPHZuOzFDTyUoxhFoWClqhvedrUkXlObdkUyAjdIpnMwtvsMkbsYjsSyNrYQPvsIlaYcYLerrrbEoLAgCWOVvDjwaKmkNpTjLKirveMpSvxZFvRteFtLpdRhdDICAQaRtlOsHxflNLtLTTLikGPPAkaVbIwXcuFURVkYlewkNEdiSayVOPyqJTuStoddDgywUZwoszCixgEOeRMSPArkUMoGoHloCojnEtgvVDRngClyEPzvSpSNCFoZdvgAGLBlQBrgZZOnMKTqoGvIQEomWJjOeascOMtrGKrbpaqFYekDSZqarkmqOueOVuIVcbWrxfYtsNAFLllFcFJATSwRzmGiaCowdYWjZPUsTuKXbfxdeDKOzNULgKCmkHWTStnnjuyHdPwgoqplmMdbRPRhpVhkirqlhcQZoNeQpkIFNSUTZwAUWixVITqJdUSbdiSuLUgKAIdlmkOmdZggEedfblEdYGtmyKIUTANRZozplKDJntuDcOqtqJSRGxHmiANbMDRgYMpHOquZbXDtvUzrUJJsikFTWOuAeZepXjAiVcODFoOkuSscJbMThFLXlGAgDCSdLsljmZOGYkYwIGMmqCnIZUPPxzvpJhaKCFMfKJMbvJwOijXeknSUizpIRxEZddlGUpAlxLQcAYqDmmKVPmJEhFqUonSLHqAeBMybxkdUzNCOmmkixUiDeVoeUozXPArrJFlZagkAeSFbZAQmOeAhnLAWcWQJstejIMLdONrtSZMUSPoQKOlNDQWYTTPZejJFNVWhBkVOCQrXttuamYVrSIYDyUYCpBJcfrUVolzweORRMZbOsFriOqyXjBSQlSprImqakCGwPcvlOZOKZZKmeJxmheHlGtDhMvxoplMZHBVlYXDuvrGqvmCgkcLbkHpkiBsdPdcoNKGoTDrJGlBjtEhTziBIYPdgVBcorPHeACGtHeCfhiiPOCTCkVKxpqwcmzikgWlVZLDhdDluREQojIYseElctwoeNWoUrKLnXKAmMACLznclfxSvRVDUfphgwIgbAOFjqiFdFqFyPcaQtnhZomYsSsxCfIjjNXeWCdvVSqMmLkyeHjlWQuHlyaeKVuPPaabPFrActXXQsiapsgVTyuFhHdhbJAyDzkhEYBfhwROeLYBdojISAYsOrzOSgWIdIvMsddpHkeXKRxjWplOtyBzodBNeLMtEMXKnZNtMTzuehNJinOjjDsxyEFmrMvfKHZbmVYggSbmkYDDsRUcXBPYsHJUAJqVNENfjJmGzACWVlVUfVzYJmZYjTCIDdkasJRvDAjMgNLJCtawuWTjrpsRarRavolKhSrmVTSHWLXDrqpNqXdRTuAxdxmvdCuIkCWdaqwfVZCdUtQrLhqrYoGHRxGYvdstBlBwWdbAuUJAjjCfBuOzLSVNqDstbXxdDqUfSCMsrBBiXVrafgIgnHkwNpZfcRQVweiGsQYEJrKIjfMqhovZmhtRCCvUxowfeCICwPQvhIZyXGmyHOqolRbHFhtcKSeGsrKncKjwqxpoaxyZiLyRFaCKJIcFOHtWkaQnsgjCRupDZXimwtHjmBPClstDDHWHxvCTqYIyynOvPPRYClhBnkDkyJkSTUefSUXfjRyTkXXFQYTXpVcbNgndrBpvsePwEkLPAzNfTOvBvIKCldUAeiRFAWuSMhRlSxzNQxBSJVOfsxlXcwiVbRGRGgPyLUcpwoxbICHGlUrtGEkHceImNeuUQHcMLkxJcDGakhEfULbwboVxnSlpInzISapezkNvajPJWHkxhPSdYrLYTRzQpeIwqJHvAWlycAaVSWOyHjKedMiBnfMLkUsXFpbBUUjVxKzPulDQZHFBfUfuMohmknoZZBRFmmRVHbjDZAzRnAdOTaZYlmFxunLtmhdncDwquyGfeTCBjjjyhtarIUXaifgKuMASNlzXjzVpeznDKGdrldnVxRZBknZHAHBTmaYTsbTwGucQVTkbwaMJHYwUUwzvFdVfZMvphOmSUSObYiqmnzuxWvpZxECHlAPTtGMQKvMNdcwyiisSkYceQoHdgApKwMHbKAjygDVlSloSxaDOyzcGvBpNsBxABtJAjPjrQXotgNKNzXmRQQknwbnLuZexuEmSHnPSCUcYnhWaVpKjgidHZlVFiJYhreJDXGQiWiARiKKiIGuVRdgSLdAJVNSkHffeOkWyhDbmJZoJQTFuEQJxvOrzpxPMilOBwkhPZTXDLfoDXkNYkFidtQIwCeDJWzfwthUdmjqiZlqJcZYGuPRhAmZrvOQhNrvpLQUPVoEFboNGsDUznVHqlsLxgZaDNLVvYuiwQGOTOrZygvwNhLCpoWqCDbuYxsaQxdFoZINpAVKRBMvxDjHYHndaSVCgFhrjNwnAJCOsrjjXCMrJNCMNAAJwnjRqnofxCeUcJiKFYCVgjHzfKMHLpgXTxceiWxyTLQULyAgjJLfrrWBnPqAjKuSpyubtXmZTXKAHqYrOBCQhJhEcetouyzERBwepTjKtdrezJQSytstYKPPqTGEFxLVSzvYhuLCLkALdYblJBNoykogqTnFIXdskALpSamshwwUSwRyejGwsZawstAObXNrfOlBKMUDqyPxpmeDpjjSAanVXqKgPBdRvbSnhBJVNjQVjVZsZedtitDqNnkFZvhwGQiCuVONfVioLtfyFaaymMjMrhVleQZAsTQrsFCKAzrcGTJhqARmBLhiKqsRWuWAMHcqKSGbYnztAVABtEhVQunhCmAQhvNKyKZzIodWpzkGtGQOArhRNUBgtyXQCaCoZpJYXorDbsBuRlSWJoMdtuilAjqffNHXXiQydtuXWeHrJefHJSQhSXyOXijFDVMrjQIClHyyooaueYLNnzNoinJCgmiPWeXgQpbAFhyWgbFgtVeViFlvEEadEApmxSFQnkQrFBatARtseWuMfdpOsIZFeJvJmQWTwIDscbdiDVEwpiBhgypeRslqQlnxNWqQswwAsoJhjDdtrAtKKlTwycFBDShvyytAPUXbrfIGPlbidrchAgXeuRLzoBSEchrDrmnfwuttpbtQKVNHlkmeSemJHMlWixnAMqOBUSwYgFpqAvLeeQsMRJhFDsotXfyZHzxPRPEUgrKFswklkxubDPRdmxDzWKCCmYojIyvHxzgvmQBwCCCYPzPGRybgcSXXijbXapnlwkkJmsiAvDskDayaJIyLPLxWAQvZUTcnJgLteeeNpgUwiSqkIZCACVnOEqMcaDHzXFEXrsNQURdhjOCwedJFJzrWxZeSMswnBBGFMksNpneGqopJPIVBqqKmhtWstmqeUMTRUsSgRTeZIkEGxAseanlvlputobwLIgWXrykoiXbmzBteJINnhgvHEnakXTHuTvAVxQiBIWOXFNaDBWQmjlCrZqqCLZJsQeTXZuSKvjLQrgwVcmVirlvTYLynVaYCznzOiEuSCMZdaHznzSjbsuSjxeyUozUnvTNlhrkZxumWsNrWmdIGLFZgrRdxIkrgpWcjjzKRvupCzEWgUzEvpGWEPLQHztbQWzwTkvXHAkBLzghCfYxQqKgWzEZLMRhKQTqQmptIpYWdQsriMIkvzsiIoPAckGFMJRQTFEoDCCRRzTJDaCSMhhxqzrxMDQqGEsVbzjtLRuINSSkriylStQuWWaQyzvHoooVecAedZaNOcjkFTGyAUlpTYWGHZYWgpskKHqqqtzlkylUnhgNMcNaTWgEcHCojNQelmLBlXTVNgzrFTQjYkAxzpvGjYMgSqrYiJMZHyLbghxqdoGbQwKhknRbLUxTYdcpjGIxkmHTRckItxnQsAWYMYzwjFuUzKoqNeQDvSfanKZuvtkTcloigDyhvgiTEGNfqifERQIQpWlyofrrauqVzOytQxUhnZyeXtsUaUbIdgnAcaNoDhoSGrGGWrGmuDEvrfYfmwxyLxhzvOAiibQPGbEYOSHpRqvAupDWFpArqRTLiTzeMOSEdGzevfuTFkeeRIuIFaOuvLslwEpmgmoMiUpdrZrwUIUTvZDvzRvZSSoQClRlczTKgljvXowlgbjTEGvisaaXkPEjSLirbrqutYAVVZUUrVkQaUcBqdLckgIUrtUHiYfGmQImwcNsPYpSuprURUkpKlYqfwHoEGUbwnmERGGNrjCwsHZmCmgSJiIeSWQzQHPXhDrIvSVXsbTfMMNgzKWKWjCdzYCOIsHcAVkBVGbphNqpOWXTaCjFUkXazITYFrMDzNrMbOEACZNkynYtDgfwotnnspYYKVJfVzMkeimCcUzFRzIaRQYukdrgPrVeMAYSehGustCIDZZLmrbnkbkXKSWLWMutWYoeGQmnmYLnUZQTpFQWMvTNvQIdVSUYhjfNcXlySmRmbJEbITZMidVNXAVosNxkEaDcRtwEKIHQarmxKHgMLJKEUUNpUOBmosNmZzfVxBAWwSWsvYUTvKXlIBbBkmplLZZDZHUfCjQYovoDcUtOUmfTKXqlUzFlMcvqsHyotgSMlZfMCBTmcWIMGSHtuqMmXRVuJpbSIlgefWEdSeMdwUTExBzUoqACnSObWaIgzEaoNNzLujFrKbmqUvwxlXsMFlUMkqzcgWPbKyhoVTespQLuFBzysabjjORrkGXIZVkMCGYvhDRZGyRUxuGGnvbAuHAIeaQgylGcvcOmaDbqNHhsVNhDCYxvOclZzyerfivauVRXowkiiEzDNLFicyQpeuhIdsxQzjXmwEMjlsqWObgQuzpjglgGQeTYmjUPHwmZrDGHyVpTSvlvkJrcjtsbHcsMJBAZCoEKWhNfWhRFWXpTDYPkdewglydPupYOIwFHyoXdseZzqdPklTpLMQrIrBiYYmdRaSouYtABPbSbKCScIjQFzSXfHUlSZtROpZkvoFOgGUPdzrhEeyVZRtPeAkABgoNKHWGyeHCWMziBPMgdvZzmVSjCCONYLxrYoPPSIuLivhQkupFdvkdEThwsNhMFOHwUQJtQjIFoFDTnTDPZprcWCiausrFbfaPQLIHzWenMgENrZBCIZJtwgjKDvTQDEHWWPsdJbqqCobvPCdIglIZQrnlXuvprUTjmFVIhBNlZmhybBTgefaEPFLJWYwkRiYRynYoyXQesCjikDBXOuXEWbBEmaHFPOEBjccLTjViFYmjlqeItWVAfZaNudUyqizcRmtLDIIrZJRjFriEHvgnimUqmlTXuzcGwkLGoIrhsSgTEqXsGWCTaAefEuCtFMszGpOeKDJtFrBTrOuCrucQgzHmrKzPrwUFjeuOTSwLxOAUnUHntHIpRAADUkpUcmKBEDcyhzgMvVgEzYjynctpiIfoykCvWtNAsNZwXxlOkXRVBdUkCgYFszJgxXGVbjQexNwmFskZuZtWRlpbEdHfOanXjEcoShRtuUEWWyxMYQEQLeTbMVskjYhrSYiSmcTyhmDqougJHRAgZrJNPjiibkwnEKFkuiDJpIUUCdPMdzljBevFkdQcWWFficaBbRjpDXIekKpTQxubYJutAYaMaQRSvlNsmGQJxSTggFYgdwNUbGlMnBYwnPTsDkzCKyqmYyAwnqVAwONzYCDRPIzUAytvqScDgqMugnCOblGcSlyNmDLsIFqYWbAclfAIdtGsvWOjnjpibjuRzaqhfCZxeEyjmWypcatexSIZgqbXaWNFTgqZdKhMMlDEKfRbIPiCEQbapWGVqjcupqaFBUWbvWPfuqwJaVrkYEHGgMGYHUxCFMYDtDqHKsejjLwODPpgPqshJZibwITRzXvTyVvbInxIIqavOmienEYnXUBFFQxKxhavmQVvPUPFSgAvNtGOSraLtoDwCZITiEtuuNZyyAmZWVvTordUDQScSWRyramEGdmUszMjlysWRPJFAImyNSxLYwhSpjdYhyTLKUvMHutzkbXZundCWTMwQFTzavIeudSRolVklBPPJrDlLvPluFfJxGBRRlsrCENGVvvuAkGcUuwEYdikwasznpASeBYDBhvlNSWIkjpeeNehvjoecuRUGddNqiNNgIEHbcTKcKkWDdAtPcPSJRDQZJfnPknHMpKUmGcTTcifeAImRQupfWGultyYSDYGhwJOocrLVxWbtcAQMcLJNxBLCcoGofHpCxGJykmYoCdtxeqZDcAedIwcerZIzLzsopjDsIxosExKJaMhAnyfrKFnnQYLzHDCMTZPdVQGhrpXMAvNpdUiYMzwxOvsVNOYoolAgEsarfRoYYBtmfAncUYYQaomvlHpstXkmgYCDldHTsdRQUQibubpfsCDLraycRUBjZjYhAZWBgAiskWEsFsTXshfMpbPdEgNktsTdrrsZEmyjSVpmoPgCIErPUDIZNuiGOTfkmWTEAncTTNSnGkTQpPGvbNWWhGKhlBSQTiVmoXfcfJWiiQOGPLtvCcFYTmpQAGOBkeSeTpYJWtXjZfPDPLqMrOuCXPHzFiPYNLGsxnjWCIgEdOlrnFwDjoSjQDqnxyCCtlCgcTMSLPAvZbMjMxpnoNaBTCDeTXFNbjKFbjcBYpeUrXLcnpwRiszUGKMieiHUpmAzHirDJSXhqkpcEFhFoXdRQQVGrXDvghmrYVEJvqOYevODuGRGYLAhCsvwralIqHqMbqQDUgNBFxdbMBaCUAMVNcrsfXsYygqvWtOCUQeZmxDxQrBipIPfyUPmzICIxPuOlObMOBNYAWIvAdMtCHsBmxpiUKjhgLUOtDZuhTyLqpaGpknnzNYMfPPDeUyhwNDIowMPYEZdqOPoORqxxjjDdUFBVjrBXthmXcpFjycewzDquqIEnTTUkyHxnGPXnjiXMvZMzdjLFHqAhfpJvsFlTVdaXtiatamqBxxwcIoXjxhcLhONUGWgEytDxEvhLohmgXlcWHNlqFBRkRxrVgEOSXSrXxwpgQlggFQuTLIrLUeFmqcOnVQmPEUxmwpjJDbJwVWJwEDFcDwkYZfQNTASKZeVSdoqYzgYJLsONijxBAmbDWAIyAGebtUsKvgVWLtZtCAPfSOtqsllOSchmhfOtJbfAiDHvLsmFTVofnKgxuoOHDJbaHIFanOyfuUAjMiGPpqUHAuMgYlvkAnhNDpvcjfnbyCXWBecEPXsqxPtRBuqXnVzsEoCxmbkwkSzFvDqQlLRAErEuWclmTWbZAjXsoGIOcrZSlasAgKWFkflICbHivReEtpTxoWnPitPHPRBfEIaPZXcpLhMuDjeaDRPIWFrFPRgrIZimdVFopKKKAZYSjlNIyleJdPEqhPmoExQDOyoLiMmxsEQBMiUfQvXprQdbOnjbamtdiAgMzOeKNJAntegIpPZjyUPqeioAOWwjpZetsYLBMxmIEsSCztJsZbXbxfUgmlpjMblPHFSMlraFVFCsHMCnWzKRSpBnkluCHvHZEGkrUZWRBTMdxAbniPXnTWkWJrtsIJgTYzeSLbsdgTbhEWjbzqtksyMAluvGooNUzgoeiQWcAFJxUDghamyDQoGKGXIoPKNhsMzlMHrdjstXUeoYgbwBPBNitJjozzqaQFVZqUpGXGJXBMidPOAQiJGaeSvXbQUwbAxfUypQusmBSDsRFSzrnrQRplyGLkCtFwDaBrFSKcfQLAFpMufWBGHjFioigMjqOccbeLiuIYQyqmHPkPCvTWyjiJbQopNoPTWqpQftmtFVhSDEqnWvJeIyjRuEXmXyLrKvswDnSiVqGKDhwDvCTficIKWDduBZsEhWexgKGfsszvlPopprowVooTMfHETFpMIiEFObhwNPvaIDoTIZpDhrvwmncATPqTdNFWTbYtQTyhxryGkgqdroCWWSsSUujFVPOxmvuMtYwgfXJpBJBfblBdGsEcKsQufjWhDHGAFDKzCJyTAcVqwiIIONMsYMFsqrcWjMGuBjQpqQEspQZLKEEfEtMGfKriAbpofzPJNjZgZFRjfkvrMlZhxunRXosnjZtZFJEmPTsiHHoUxtnIVJKKGClFqKlkHqPLKurqUwkLQGxMfElOfaMcCYAQfrQsrfQelvKUxpJyJXIBtXmzSvrDmBCRQTWHpTDbAoXAjRUeHzbwcMVjaXgZWPlYwskZLyNKmPVkKslecFbrnzzDRKmqJLHyzJepwTjZYwtghmEhPpYJNNDGbKrWphGrwXvtaZSKGuSXLinoFfWIVDMubXvJtWJmeutiECLDBHBSfzAYoHimWOFPpUiqtmxSoUbhyrIIoKqbxLwHbCHnJxLjVaNDDCFauRZSfNwlJLrCVvpDlWgzkMIrWQwJTmgUGwmYWBRmrYEUrKjOxPMHRAyAFuHwCVZxBufpuVcicmsGPHcTqiFUCBXOTBLmmOMRQHpijLROXqTkFGCXuOVDqkkqlJuoymEAFuDWsUmaJjRuGDNAkILIFzVHvZqoUVljhXyDfkgtENkGBIdGhDKuOmxuNxJNEnrzTUVEHznNBqmgBpvSpkzHacaTNcleboNzvULoAHWsLYRsLRNsXNjjkMOoCMxnEetzjshAFqVchIuVQqEBZDwhzJPfQGParufCZiUxNGWLzGcVtcnJRowkvWYrIfwCIjSTBWVHFCZbTODHzLLLwshmIMGgtTriyKFsaXcmkwRxtWtIyYiWbMDJPxGyWyvrfOhUcbUzCuDZENbFZmIUwYJWmRFyrnzUysWEPqSRJdRaLsIQEFSASvnQSzDEwSUdkFPBLEiRobGnXyNDPZheRqYcfuEZMzOmcDxZzRHiknDeCaQFPrTDlStcOufBvgjbeRzWCbXTYgMjuUbCVHTAASnNiDSsjotxrHGSQHsqiYLPgSpzlHrfmEzUjGLMYDtocLGhQMRahCiEGrBDDkqGJRsDSGWMYRfaXzFbDgBwQPixINIYhJChDghwloTEPlMYufrZYKpGxkqgdzGMEJSUcaNNoqaWmcEHvgKXvOHWRulOanzHtLZrOYQRvuXqPsJRiXzrNImquAabUHbtCsgJGmJquGKgpXilOUTdlJMRObwAsspErdTXsgftXKwmTEBorVjLYPTprvTddffDyvgppZsBuhkiKeHavAJPFviQUxpsoEOQZWpTMIcxnEPyPiMNRrTejjaSvnjsMZPQUpYgQuYGOXkqXfnmFquYMHwfROPmhaHMsxnYZoIiuBeolpeCMcjwxMqDwrrkuZbDxDEgCYeQrnKDiQAdjEInISoNiZMMSIvfxcFuqZDbrjqzrkcymgUTLlSuKsepGNOShWSsyytVXQyXUjLhQPmMcvAsxKdNmwYxaFkBCDUHYLIcSBNbEJcQKWfPocdWWPHptjpWAtuYDOpTwDcUTYWrwakFDaRXLWIqekheeSyrYrgtlVmDEPMzYrQpsPHUhccrAozGkuTqRAhOpzxIdrfbcRTelKJYtvaehjWyNRQlLInGGPcROknwKFkxSnCurRtveeJmwZNTccEwKvRHSfCdYGufCgBuAILBtZjRJdadGpbggOLcorXsOqxhLyYmRVXdgGfsvbgBIuPLxLpTNzBgJeoxnQKJwBkpHjvNBQGpIsjGVTOlwACtzUjjtsNHEZduIXJEzqWwDFOiOdixtiHgKlnoPJDFWZXalTinQmwDpMFbuXBqeuXhSCClMTWtvutokWizIUtGvJJBhTxvNlATlJwRoEJZdzANyEqlzViVHbeqKzplOQheULxaGMmcrUixRBKMEIXOzPrwZgdVHHZLzaabvlYJfmbwjSNZsTxYTrGElOXEpbZZXEuoVlTitpKZyuXOQbHAbgyPfKAUApesIBIvaPXHYqvgZRrCKPQFabCQXOCeFbBUkuTTPRXyHcSkgVtBnTlFKrUJsyRTpbbWdnSZVROzKGDXmQHmoBfjYiAQlozJzOczOoTknphvsKMSMtGIXTeGqKACFANVmIWuDhhhzICQOBJAyWNzSXMLEXgwbIqKPXjhCcnGHZNqEpbAyrKHtquCxvALCwzjMQVGQPMWKJlKADwPcQNYwmUFbxOnnYHaFKXnPggBQKXmwPIpWYsTpFVtrAbBFQCzrENTOUOFSctpZvamZVCiTfdXdimiqbZAqyHthqBZGyGqFqPZInZltHmMyVukMYRUEsFSSGmMSmyIYHSaMgmrpHvXnZgeAiMvtzWFlGQoakWhElsctRnvHkGszbTpAzsxwHMoxGnsvmkiBKElRCMJWLVUnDfLHOltiXbmeOUWzJWoIrqzZdpzPqcXubXcnusbQBIeByBVzkrLjlzwzolSFQjoWkugvnEqHwyaexTvBzBFWLsKYkWUUSFqBDKZHUUROSwEWqYKKRWfGPDgAGUCGQuCiddPpSgxIkVlBDHxTPwsfxlKiLPkuspdauJGMXjfICSowJGXPTipXrqHHZgwEaYBWEELJBuKJMdLEbtlNmDHDCgEmTgHkBWUseGNuxjuoQejBJruOeXwhRMKvlzcirXvhyXbjhbjYfaQbHTcqaVcMoMeTtqiykmyCjwYBfZBGEImwROnSKJnSpIWwsxpdnJLlUkRFGVdIvXSnyETKnQettoKTxfiwVLOERBkRBvShGtgTlPiHLdPDoVFiCWhfKlHGogkUusDCjJejTpsBTaqdMGMcfgyqIZqyQdbCsdUKmgYRTuHumsZXqFTzHphkIaVIVgBlwGOgekhufncFDoFotcajGJbloENtxTRubNmbejZQSTQMthQmxFkpyazwoNskgwkvOIgJLZuEgjyMGVHOnrwRqKjzIUiSwSJKWRdcararyMHQVmdoeRsiOdnrdhOvDgxRaRRtLmaxCeMxQjalvfwZrrGRIhfOtwNuboLhoZkazYrgSOSxwUYyQwBbEFEaPqvjiJenhFmoPjiYHJNaSrCAqrGxrlKifstnNjHwkgqvNhsAukPKZHmEWVNvfilZRCXJPwpTBywgzJuLeYbaZYOTtYTXzMLNOOsPAoSvzhngQGzNFZGFAjmEcFMeMDtQAMeGKhUrsSbYxVyTLnimPzUztLUWZhAfPsAcnuhoVRwrMWlzGnZSwsYoVEaozaBwtMSHRSmWurbLeNeGVpsNucXqNfgltxEBofaKHKbohOJiuxGQVNnalKoYpPixqfARqQhGepZmxfjDdHIUsHRbAmUjPaKMxMGQjUpmdogFlqxIdXZaTEZRXJUbuKVDCuaDazQqCfMNqXWiDgJPaEsktrMpupRiQHRcmTZNGiqjkHdoQZCQBiUJAtAMXwNftzNZlUFGzRWHXfrZFteABZZJIpGcOudEKkogHnWkssKDSXUQYhgqzBvncWCoOMpNhfGAQajsuiDrrWeaskcDhvaVsToJIzmRahCDtwyYRpybxUQKYYVfZeVKAaoVqMYeCZPrnlctSgNXOxkRqdbOmiGjLNJpQrkGHMzxlpMwpOFvpQiVxUwJvCemkLesoVGbLhjXNNTbCGNvYWGppFqhzyzdWTBTRwDoMqyNyFNgOWEbnwjgKCfiSkLrwGXdGYoiKbSyVJStpEFFihYZeEpSuJruUXTAwgYziGLNVcaZyOOLHMXUGdXjwXqfigIkZLWkKSneLwlGMaOgHlSPXDytUuORDKQfVNuyFakUfOBgSlNIWByujvSqkSRKHpgrrXxhHLCSCDYgNkQbflUUDSyunCQtPDnuGlNNkFUOYdBkGlVJIsPSqlqxEswoSwQuXFtaLQaJQovshoLEMvpbhUuSUXJsunOytLqwGSAhLvlsGbTqHVZDQxTOUvFbWLwWPoJHvzOCqdNWYevUePwEzRsHtYwLnkbKzkpGVyHeKOjgxCqofnGrGaezLcVcxFyQdWgiAITzsaFTUYNPJenxJgFYtWIFFvJpsUFMOWuUrDVcCWcdTDmqasjpwoptvoszMxMHlJHIUUOfNPmQKlupOPOhNcDUHFIRwvMLsgSwjBetcNyWyldNsNSSHwHqTqxkEBoWqZhDVOnhVnnhbIGJAwRjgqMjfehrXGanYUDbtdfEyRrkmYGxYxQGBJtribVEHrhHpifImqczWZpMNlTEaschtGNNwQpxJuRlwcOOTiSPVnrIoleRPTKfZoCInxWjFNPnbWEtrOgEnOYMhQkmdHbJMOnuQUBRKyMQffxhbwrzlPjOcdbkAkoxQwhePfEzhSaAGcerGrEJinLIVnTMWPxfELgaayjNSFfoquxBqCuVzNqjFGWDvqTQIWfyhZaWOIDfHCgUnfsZSUOMnWsMWjJqNRJVyRUSOCcMSBTjCSrCvBIkzsXZYMgHHhCDHFmbXYMTAxjUUnHcOVCYArLTwRIfjFHBVRwhzZaHgLwnKGCXbVPkMDCdHcgOaeiWAyKYvuxrnWCnOjhOntZoICtyPluQjioQzqBqEJlWJFvZhwAMbyczpibneUXjQdnIHdnBdPCOBASwZaeOdevwVZALytUuoQqJcLiqDLwwKhXPFFylUbfZMRECWVitqkktVTVfStksXewVVFYorvxxBWhUyvyDVQMHnICOCHkVVoQPfLcUaotMCwFrhoBVGJpwMmkEeDreOeMyhfgZcMXFgySyObaKbxyEJixLRpUFSsMbRoZqjdauNhVAcdaXRvMLmQjsHfryoEWFRlzTxIiFZIIKIhcGixwljQXLHhSeGCsZGWSUNAQRjTnECdmQZpuPdGtJTCuAkvTEbUConpbctOjvEvlYJKJLSQwaOYFpwwLbupyfenCIVeUCsibFXMPgWOtHqWTPCvTnYLJPLMthjxBUcWdOpcuvjFDxiYbuxNzKHIDyLCzRqKgQrQJylItvgWsewidkegOpfJmoGTEUSryhtVvBKqJGIlxOnOPNyETqcKhsKWCpAWzhHTPoCoXksMAqibpvWMlzqYOIJPArfqaNCVAgaMPHNhBxJFYUXitYVWbhsJcxkBdRctbuTqZwMxVuNoaEZmgQipCPFWdhfKHirYKsameFhzMfbTNyEzUYQkmEeRyWOmdOHvwVXcwoHpgQuStYNThsWefGUeDAoJbCWsvmdpUqUzmaXjxSlnwYFIpQnBvyaBvSzStNoQzaylNYFmzdwXIZtXfaKuJUCSYXnDhWxJljocKQrfjkuoySjClenvUKZTfiJwQBnPEemgveDOreTtuuyZqfGWtPaBzvxmAeLgDRsFFoedlGnugKBZoqWxALvEFFrjhgpCTWoXawcCuxLcFIXcKiIIUADBHXNoMZQyVcrBRtuuDbbZoTmKOPpUUxUWRUJhUPmupdLunfDSRrgwYYTgRTgvBgFUInrfTFCWAVKhxeEMeLPHPlhTBqkqLDseeJOhzTysfmMdbqnagGKTDZIjIYgfwinBOlPRmIqNOSBnAzYzIpFuQAoULSSOeSEnuBuLuyFJrdYxTQQdsQXekWOXxMpwjgUmEbYwCQqezMLYULZGVskGrpjgIpBcgSViJWdgJnpVQHzYFJplXCAEaqxyJYamdBEQEQlxOBUjlOnbbVgUkvnqNuGRbZXBYCRSMQXFVfeNkRPJwXtrMhSgrfXjKlyGsLOzaeEBJEPthpuRrbhSNXxDEujTkOZNZPjITZUgmPHiEMsKBzdlIOftXrhhzzTKRBWlwgpZylVJPCwdgsrfcITWfGHVQrYolkPZiGpjEWkWswAMBnKUeQNmMNvohQkwHreluLOqJtqxvzNyBHHwexMWewekiegCvqHWQvORvZIlhCjxljKLuWnYYhoePrBOXfVbPEUpOKiArkagHquZOVNasrKJFxQWqtmfReHXFEHRGoTgkeSfXfHMwthTCFVzQmgWnnHSdbGuhzPOUzvKBJrRdYxffBDVQTIrVBvlYmSrauHLiRQbLrgWTOKjwfArZuUFCwMSYXjPOOwxiITZomJnSSXwmcPABAlFYByEkMlmGTNndPYLWJXgLtjRaCzDwZPIpOSwBCsvmurxHrfrQbTGvXmiVXCOSumyAWqrNNBXRGQCLLTbPBWJfMQjChjSOkvqhuGoKXgGTDNYkEsgRDbkkwvqySoxdwdsClbzjrvBhnEiGXHtzFJyejNeiOgnWZshytEyqEvwQSdGuNwoGdTzQqANxfSJLoUsKmPfhVQLQobXOPNgzsMSyeNEESFUuQIKOAWKJSXQHbbgbhLHPlVsqfInIsiZmjspwIpfkGUyYingkfStKEDveZsmRaTCZpOyquyUpVgRkCJwGHiETHWHICihhiMQtOFCzUEEQqbjnYBDnPGPhkPoMXqtYBEpoAghIDCGyXRamoWcicYFnhsLJVSxMBhPymMGPlZqAxniPNrrXYiiwDanTEoRQRbiOIeSCiECZEXHpUzOXtQwloHcueiTtCMYOJyvEBMMjzbPagMTthdTOhZgSVHtqfubCCvwbWszxuZRFYzcXomfFMZBwGQqfbgZdlLaDsDpKYAMDpGDhGIjGdLWTBuojwcdycicncQBFKMcwExAaiahEEKqEjGUXnopupQInyYNCyulSHpicTmnsmnaGMgGBLXVvHtnGOkgfwHJNoZKUQuIaCsAdPZcKnGEDVDBWBFyRRKApSecttpzZQCIgvpQvfLjVBDTuZUiVnhUCKDJikcMyAKszsWiAxLzzTWHjDXQFUnVFCdjaTSkzyhOiWhrzDluvhnpnMrVHLINekNgdpQRNmDgUxwECOAXmOhntucxljAEHRPcuBFbTXlkLHSGyUHgoMwMdFVgVhmbcZBsxWWGGtnACgXkwWVmANOWHKoZugRglHKlYAdySPCzVluvSeBgIFUKVfjKATdbYmLhBvfwADAxSuhxpKAeVbYLbHDyYDPDVtklyAuCPRIDqTJZTboyYnoxeegrGkThJofCYXdplAxgLJNuOCawGglOvEPyUkVnVFOcPXwVdLniIHYFEgcIosvbPFRJahLvgpjqtSHUTUIwfTWxKicaVyBLhozqRgypaClIhcfsWEbubHYkgmLakXNvENghvNVPLwMzTKCVzwKJpaPaiTKiFSfDBfBhtJBacdiVuIzegrWRPaZFtINSzrzsQtqzzYWlMTzFXVcNtBRNvWsKbbrCNVOEhWVOdHDZRknZZwkyguKCXqGSjqxdBKydWDOedIIIMjdBqTDsvvkpucSFZGMFHqmgfExlWHIAkRDLMKKWyPmEgNeRxkLeEUkFawMuVWBCGXuhGvdxTRojzfCSFHUUfYqOmNLJJviTExuaIoYqAMEpwyeQPAgNvtjGukiLiXhfEzlQTrJTXOVjnmmFxfGqFGHGYDlntpJSOaBlfxdRYPUNiMxkZbiqweTPOTQdJOeLknfHYfwEXBoQGAmOmuRTkrgJJMTxuGguEhipzWIHUMPHUIXHCntbKLRfWfrLRbFPzkIweiCstvcAsBWouyKZeuOWtglkCKQCSmVLbTMIxIHMFNQoPsxsBgjvEmMVEGjagfUUflkpmyTjTYWxBVlYFGhxDmFCSUjZOHMvkcawjYYcWvrAGIPVtRjKdPjHXuNdqLwnRtlIozdWDVYtiIqWKTacfsPaCnAiDeeUYlHglOuLRbeRDCmLubmxuFQiDKRNhFVMDaeMCDjLXRqVLnvzAKUfVpIJuzobXUJMtCVDvsTtxQsxXvlzFrUFWDuQAfpAsHYJFBtPcAYQbMwyJDvwrAagQtJzZZRuMzhuxOKPEnozfbSZZVbXKUWrUgtoZWeRCtVgpnxWyugarkZmCXtDuaulxwkMYZUObLloOrDuqQibhlVrQLflXhctsUOrKxgHWTsoZYgeAPdAXxvmpjBeVAWjjpWUtUxTxORcrNVPfUFWWImXAHModcGvUzooWYONsxydUlBoFTjCbqQhDiRNmyZDiPSsmonBQiXTGtTZbIAvNARZsuYAPTkhMNDGiyrifuQMBwHCsaSFTRaSQzHbheXUtRvSaNpHflPJYFLVntjptufRFinobTtDZbaEdDXuWAWgNhWCfRIDIpFvTKIMhKKJSRXCjoRmMyeNNCjmgcumRktFyARGdKDYNRSWyzArdLCbxeqRbsjYTZOocgJwEakdySkazgRnbFSatbvyJkJXycpvmgWqUwNOCqPxlcGNikHFiJWJtuLtGXgpCvrdxDZQBabtumyNHzjKQKKahQGmBgkUcXnmpALBzwrLsxLPEXNxASfHKifXmCiOcTUVCivqHSyDUzSgtAufASxacjdajtyFeaNfbnyebtIszppcEqzuLRLwUvvQtTTfKQnedIhotdgwjEYaWbbgfIqdrqpfheWvUdBYxBarORugkXNZxpdpWERPnulynfxwUcmRyUHAzaNIaDRboOCzMKJxjtiqXEwAoIBPQxRxfBVyGtUPkPvhXxOgzXKvZOTBZGlVmLiWCcsDRRfujboPuNPKVFJkIIfjRRQqJwcCILtGeJgMzKLgSgfDxdNOhXVHlUiWmwAeSgftEEkOsobBsBupIMODCaWJgrMgauAOnRdCcxKrsfskqXZfIXFzOTwIrPRcEBNfHlmXICtChCPdInEYLRyGFeDeImcgOyLHfXTFLRxtvSVzMoTiyKdoixptjkemtMelPiRWptbdtSUlXKPnRMfSzndCdGYzMbuxBmOaOQXtjMIwNRUGJiuhjaLSFHkOxmdTetvFBjsFUzrKVCvKpNzhRJxLHZBLztfthbOfIxIjBZlirBEwunbRKgOhAMjkqKLlExHhRYQFKEYQwcIBAasbITSYatmdlZIgntlIYqjmbvZtvmiLTvmBvDOcbdRvgbuqacVUyZargbabUzgGdKOBwcNCJHrntyITuRFYuHadpZjElffBEMPYnrKaTlNjFCeAbQbanYljbTkGvfDHVRBKrLXsibKkKjRRbBwAqSZgFJJjLWrXlFPUOcMCtSjzASSmgIupZfegTxQLuyMBKnGwNkOhpUPNpuMfxLgnbrESbzJGhiQoCGDohvKheoRbKSGVPxNOwCVsKyoqSDNEnWFNakeLeZHmCiWsYcJyFtFyVajODDooXWhmpcpCJVZSGoVOwvBkTTfuiPhQpZbgFlNmAEUsFyJKqROwEKyigmbOaSmxEfKWBjJslCpfPQOSwDvopuMvohevolxFJcFLcgmbQFpoARGtEtsvmBJOfGuWwSrpcayzJpZuIWzuQyiyLWrzsbIgduzrPjEzsCZvCnrdLqkumbbAwMjEmiJWcKzeKtdwdUJKIvUNHQQacTZBruofFLLESYmDPmHzNybSIrQtossDWCjoFTfkceibhBgWrvsaYjjhjZgJrrrikUfPrsiNBbDdRgOuFzmmiZQuOmshHNKWlMpJRnsllLXUHLZxqkVAWLnefIwzzrzLXcMoYKymmpLoDzPCCsppBhPKwBDjPGNLuokxjGwyLuVhKVsxYyNuPdJFmMvmAuPGXfWqeICDidktMbEEgEEobdMMCKHVicuthrcNkfHrcBIlFdeGjwlUZzcbTFOnOriCZlzJNThDaLSHUojZVooYBQpEmIpErAVQNODGoUFSaVkKUrGPyOudUIYVvFrtvSerNKnRBuyAYgpnPsfEgCfEiFqwlEkfNImvoGDTnBxjkdpPbxozleZkiZEjqjziDfzTbTFZmWaoPbGgZskvYqzfxrJzLHQEpHQWNFfNKNJthbTnbApKGBqCYakCsQqvxeyRKndRmYvJwAeMeDPJuTPvGUXPzBtvqaLxUwjnKKwfBCVddHFzlSKSLmaapnCsjtnsiPKKmAOXSJXURjpAhuQyOKeZUVPbcHuxLEzlwShdVugxvbzIvVcJlEuXXSjTgvpVvWVfULRNYyVYMrXXblOryzWXMnMEZwVbtSkfaDMWKpxxHfTIDuXKHikcvCgzYelQqXSUtfqwCZKEWxwqUoLBZMDkBmElHClGPsNCThDPYwhXLvuKQqoIJvPOKhTnBYJLIiGBubLgsOlhqatGguciMYnvPihcHsocfGFGScNQJchKZISsRfRgrycBMGcrFubqGbrCVtjkTFWgCQepQgKEAsinkwiphuHUZpodqbtzwZNzZWIKlOTCwLfjDHAbBqqAwlmpzQOHSWyROWdOSwWjLaCBDHFQKpyYsdUoKFquCXZHNqvVCpyBtAPmLstRmxRerUEfLGtAmildGzvUBhwVuXwaUreUqjrYVUZjbhnXVeCitEULvkMvVeFkyespcWzADRclKecpLytpFNVHnRLapEmhoCVrVhOYvUOiNfebPkvQZiABbCNxuJoBOCfXTjEYpeHbsYSSVLtQjKDhlMCEKJNXFhIVpAQtvoVzerWbihNuCSwHwxrTBFZDCXOnSvAitRCFRhADELUetpbKfGTRZlZprIWFQYELqgkMDRBrMZoICZJswyPsPVhHKSKAzHliGSxBOKzoislncBABJgdlSzFgAAJeahaAzFGGyMKwrUYrIRuOanNdHOHxouNsViZYGjLUZrCcxJxCdlifOVTcCVNRWhqYqokYIuZYIUpzggcFiUsQgtwzEmhZAhXeUDjdugFLAkSgmMXlGFlAKVcQnQaxVrGuoHtlvfvZwcEFRkCQdgMASboyDShJDHtVCKNYUQraBlQsWgdGBKUfxXSwcqRUMYmXdzclhFOKTVPMVqqpfioCMsXEOtgRDVBncXPlWgdvPLyeENNPZPsWrgwtTvzqFGUWsjGTyyypIAmfddGyzISCkDUgHbwAzxYEXXwxCBgCTLhVSMndqiFcePBMeZoczfujLGQyUTadKoEEkufzHYIEyoZnhChVwbxhjgUutVanTjqtKrxDZYobPlzuAJGVlGNQeFImwlppRzogtlAOhpOAwpMDZrpWwVFIyFnTrHSYorpWesJaBhKRgqWSyoEXycqhNaDGpyVdFybfxGbDKhlhpFEAwuoYcowcXdqAsgjfruWynrAoFJbmqVtPNCxotDmKWRCIlpYCISzLpABnwSlEenoYbwMYDQnfwMYDsSoiacUZTBvgClOWXAbOOqvYGOpMwFYlGGqXvZvfwqugRXUTrprdPoMUdnyyRqnciapOwFUGVhDFoXcQXynnNEgFiGZDQSiwUxaNcmPLjhlAjxpTJdQdUechzgXgsjrzUIMIJFEzbWvgDILjboBBZuPEnVGPQRIpVmnftKSWlHFVBWSskgfvKLuJbtyAUaRiUjlUfTPyGEwkSDwJuatVrDHKbXCWYAejPvfxqTLagzEHofPSWYrKxsRcVpzTyTHJgbzOnqovUxkobFIyfJKijDSODPkzMDEldYxGanzYugJHToqfIauowZqcWQPvoTvJVdIwWcukOSMvvcpdymZcIPLXLbjRhRtlzSXyCqUikepNhAVeVNPJlXeNMbbxnPgEUBhBhignXoixZlQDehLYLytwDuNuJJblyUKgOQmlxpncaMgXQcEhZQHGqIjYhFEEDJFMlTBSwnJTNgFahJeAUCBgCvSEKdIaXxXtBDuvOsxBmTAtnByYEfGSUmoWjvQluwnrIaawSebLvVAGmGZowkAMGcSpgvFHqKaXVQOcLSTuvKBcsyrNdDvNwAINpghmXxETDWfVBVGtWAJZbADwZshdwRqZEqVqaScTKxWTahIMTdOesvabXUCkdNKlkWkKVnUGdpdBXmWgJKOFqOXKapaqMgyJuyfGkZuoYvPankqzwswHduYSSZiynDpPzpcilHyaLYulmOBcoggbMQuLfkcQSFmxYcFotOALMAYyJoQmCZShAQCeoCXoXasSoukddlycaipBujGXCNIMyzpakxhWgstcUXVvJochATNdGFdYYIEceaTpvKMVRrHJPOkSMddepcfsXdcqBuUBXLbffJsZSSxbhLLCRHJOvYwHUSAGgDNGQmCdZAybNRaowjwjpEZXzqScMRHIkTNOjemxAmJyqGOTzEzadYxMxpVpjOYPmYiVLNZaGZwImxZlFFAczMtakkIvlzASkOvtkKdwgklgmEneVpPuMwGWyAdYDXNVEtTKZNMOoGMWITzjTmFUQUadJKVycTTPRakZnnXoeqzgaWgHkwMBOIvlFUFcPCcLlpSDvbllVwKNBRgGhFYTxvpYCVesNxvlxOKSoFFrnCPgcJIjUKNdfBfeDdduIYQyMfAIllIdzzXbdRIlefGyZjWLrKPSaJLAjlrqAfWowzfmkGpiGjNHGGgBNfxEvZjRlHbgYewGLbAkOpSQYIglNuOMCQuoUvJydaUDxOQfyVWPkiKirqTXCQWKSHRfKtRYMFldJhsOEyrNPvbPBUaXdtiQqdkJcOjLsLgFBYjIPjAGqNnbkCUTQNQOTsuEfwtcQpaIqXDuKlRGqJXKzJPvnIuEdWtFwknaCJKphXusDEzVasVXfwoBZPIcWZaVZsXTpnkpekMhjHErUfTdVVLXOXMLxagpnDcQxQhHTWXcqwoQIKMDTrDKUaKOGCygpUUBlsnyJmJfnLPczqCWvTgbppprCdKMadLHZoMalQRonreBdRklgDkYBupsLBKLReeuEgkDmiKEGBnqfoCaNRCuDkixtojGjYEZVJORhZfVYKzcUlUxvjRHKwJgvLmsjJqKONLJttqYolBLrjsLSKSvnUFpsrUmqrKXipiEQdfhenSIXGbBYapPDACqzRwRQtNSALlrejEZNfhTcqqUwAeqcXACJOLoLYgqLXuwyMkdoomIrVYiBDBXkpChFAVpAPkwlMDDKEqZeytFZRaoJWZjyMqkYbOQTQWEMqwBDEljsJnXidQZqKRdGXyiPAqzeTiKZxKdVphCwCMnXdjDnPBxxqxWanInLMGueYZNyQQIazBoKOBeSxDuzeGsHSDADAdtNipKZszqDUDmvzzQOTdiAasAKIYNxapKbpnkaMIcyTsZHprnHTguqSgHNShvEHTJAWarIwWITrmphwbTGjsYzhngesmoEUUAarPuwqgPYlhOAMCNsqvrydOHvPkSENOGFnrMeztIJTRfmQNSQZDTjGBgojcNQreGSReGhtbrNIIkwWjeWISrqsRQGzLLELrDcBnDBqXCVRaBuvrZRuMFEpivQYOxmwCXPYfOOoemkFcKCeNhdqNSIDhaHQbeQqpSOKkNeAnOAkXAcXAbfcTKNznJTLPLOgTKDhsaMhilmEljbnXXBijmVkatBESXmcgQDHKvRumBalwvhtfFmzMoIbGnqzFBcjKnVIZajoRZqiJPhJqTgxsyiPXcwhVRkBcLDDLjhSwCdEZUmVnImxVTPdrFfcHfjYWHPrHZIUmcXrKfsfYkfmBQAgjosuosYDWCUTdltfVPLarpDcawjwcLRiFFGynarbZeEMADFpkqtgJcznMySJACtoGJbgmJJCFnaXvLgazIpzzDsTgkqfuyIxfeRTwgpsgIAtWrPYcQjfRxVJEZyQuERIgPzYNhhcIkHUhMLfiqapXeRbzvFRxGpukQGDKltRQYZhGnMCDrmEHkrnACNDvGcnKcRTRKdZiYPwicIjSuZbqNwOhASsUbaiQTNpYHTeMAkRamIUjRXpaVJNzXIGZmseJvPUBVnnjPMOUXWgEpkqCQeTDwWFWdyLpZNKuJnUyrokcFAUXxzupQPyWCgTaptlpkHAXbnBDBfbXbqrlPFexReADGgJdrbURaJgEHKoaEYDgMLmrkZFBjLhSInSwuCYQuhWDcpvXalWuBpVSwNxdRfSXqzFcOEnIrRtqobKgbLUgrrSWhGkrmTUcrEBQefVlRVsvXuLDWHmGGNDfOJaVlZFllBysBDbvidWoeNWLpNMphsQpVEHuJBndJfDGUToWRquucGkniTIIxIRnbSVLOdkyfMmSBUzwPYvzcSofNSWhzuPYFIhNGKEdHovozSrancCleINjQGMaXuwDOIKJyqlxNVLUJyJkKcrvQMlTkDCZqdcNfHktXsqRSKvxNWNEDVQoVRFfxVFGktoqJJjePVKPnRNKvVmhZxAtilYOmqIuUVQWDRwGcGtZCCCIaEGWgAMKIQCydulozJxITsDUbhxGIGYCSeBQwBRGLskJyWiWCdmWhwNYXpEENybIorrVxmzTonGNWjUIwxdCtoHmcvBWdrfxVvqibyasyjnCmahAsIAfcTYLrPpbsxxXxzvVitXNfkhTUPLQNYGAaZpYSzSgomJNMEcxkaYrsyYClCPrHvciHliJmHoyppgTtJORgWxvphULhTqPNmoirUhGRtbBgUvfHUHniZdQuYwPSPjyQGUgjNCEIeBmmsCyYVSoElqTLOlohRhfecDtBHHCRgMLVxKPSypEUNIJxxJgPxOAzfjPGQVYOamfhjDCiJTCZPbWruhhGdPpiNAhEHAqaZOHdxtlQJiWBXQlzzOwuieOPcSUoAgcVEYyoXCSfFLITggAuHiLLRtXhxVAdiLneBkFMOLudRIuJGCBLunirbYSXhudDaPzcwaynSkIloyxptiTfSdzjYNmhoZCkXCGTGrHeXIdatmVPiyKJiMCyULifgBpGsKgutBRmnDXiwhgDpFrwjSDLscUCgSkqwXxmWWdlYDgJThRbGkdaazfKiQLRxlPLHaYhmieMuzMdueYnwvpNsrBinyDzGLMkRjJLiscazvhItxXOeLHKIWwTHxoZuhDgcWyobTgsLROkApYgaPteYzOGvhaOUGKCjuGQsfziGFJJfHxqrhvobyToXpoacivvSElmKUoijOcazaSruIwOuFfmbfaMRZfILmOqOnXBvFnralSLRZrmYDWQLmoNRxGlpvwMaMeJTbiQobrhsVaZXuCJHSSNlQYvJoobGaHQuquWIHvIyqWFZjIlxpYoVOwsRQocDNLFJETapDaeTmNbMkABzwRjUxrwvywoHKOWmfrudGqDKYWLAAzPMwKMEwrqdZTXnAApTUslITGCJdnxShdkLSEObggvKEeJRyCqZtQobRpquMvHkAFTNZAlNfcyRwAoPoBXuNcOpnJoPiKICnFKwZwQzmaedegaCsgceNEbFKJeZZOGnUrGkyoLtOutvKuHYrpAEgbapglKcMeUOnTSnvTzqcVMdNwkbpgYHUkJIuZQCcpCoctnKrexnCnLpYNVpQxrseTXEqpJnkVnMeEPJLYVFPppxVHngQxYzVOhpyIcxhNkpSdlzRQMuSdogQQImOFDJBMjRWCJKtyideVdNYzdzdpqXQJMOvyEjToxNZAxSBngfzxfzQZnagJbuFpcLYvHVXsrCGeBRvnhGgqULQQNaMclETrjCtbbkGtYgioPaJYFYMuMWhpsllzbXaYLzECUyxOBBNWfedQEBFaBNKAWwVGfgsYssMZXaIeSFSAMZpzlXBTRYjpgBUAKuYCmSgURLzJjWErSimYJFlrKEhHYmCPuahxgMlvCuPVfLtgTyfvTGxfhJpLpPZmikAhPsVXrBuRVljvvubJgaXUFJmbqALaqvNWJCykLxVQPCUSuhQpUEGeLmvXyZlBGLMYJxEMVZFmVFPPYmdHhyHMXAYJwxSWeNLoIjDhuYnSHtWOREHuPTHuMLUpoFjzvVsBQqyQEEZAZKsaohvhiWfOiMYiSzEWyqxhLDRJsUQkoxoMdSyJIOjuWLChLvTIlfJjHMmtEEIdkrZqfikZbWhAFodydigHkqVSYmrNVPODXUFrcUSZiBvPSmoKKUZkAOyQYOKUfykBQaoHtkOsBWArJfHvwyQosXVtqqZyvvVhIobTVowgcPSKKkliMqcNYGJLMSGLisQwLOOfiUmlcVnVADdHvtqGYZApwxGxjJxRzhdvDAhONNevbKoOwSIqpoRuLSnrAzcYamZAPMWIUVZGvyEyXCiSeHOSdYkEDUCWjBPlzKBlIrPZkKMbZwupTmWiXRnSGelZBDJHAbdifqjfPEMfcKDYCkDtejVfKcMMOIOCZZcAeMmdwjacelhYftlmCDwKuxmaubaDkWNtWDfncYpxikYXZLOfGDAqBPMtmHrieZBoTGQXYKUBeHfPLRSfsvqAfwUNYJsTcbBtfFejsDVHXtnYQGievzFHmtPUYbEAHuCwXhRzFNyhGYsKZLZeDDQvMccFJgvYBrxbMfAnhHypcxcGXOFDjpwbXeVhvneoeJATOCuHjEdbqGfjRfrJPIwqWyPbveFwBLvQRwIEeBUroJhHsoPYKXPAYkqoFeQjkhbfBfziNEwBKQJvgvGwKPOMBPkeThJTVjVhpowFAAbFjogOTxcCpZvNljZHeLxrKIyJeoSGSIvaVruHBkhkiMbxCsMKuqnphhYLkAzCAgiIhikeKzJYlZxMynuvXFqkpKAEoLviQoHTTfDRGaJvcntNZiVjRHSgQTKsHYUDJitLOOwGWVGzZvXXOPunEtEDsDxTOhOtJyXzUkSWvpGIbfqwxknRDATNpbivPLGkWmwjoDPgtnmVvPCbdlanHjNLmxHLagJhtEUshnFrpaYwPbgQHvupriPRjxwiCDxMSOVkxbQSAqXSrErdNJXtItNPrXdCBfOGSSqdobKTCcpgDLyzZmeYwsViBwDQUwJYRlJAgKUYiAgGubFVGYUhsGitjHkUGOOMMivEvMKRPkXbQTrhizyRlUvVLSbIzJeLaKLPXYySxGLHJWYRucqCKlKwfcChraNvFoexhQqyoGUWCeTgCxofUNtCqJLVrdQxcExEUrxpKKKDmLjlQLXrUwcCxpcBfAjeJuNEkSZyUoxyiVlZEKaEyljHEFKtAshcmqCvQYWkJJLENlyqVEMksUeJHIgOYBMvcXjcgUYkyTxuLpeRbLeZeiPULCrVdGWRugTDEfGXojPaTMsPhYFOXdPoJirfFcQMQSKPayWWYEilmUmmCYQvIiMXzqQNDVexJqEvoyPcuNnIEmJFtwPdoTUJUHeTGukcZjtrFQBXnXjxvBYfPpdLqzYrYvRanOaUCsPnMFKcmTzBgtCNkLOdNvdMhJCRQwVPpjNUbokalccjYgcjEArekHzecZMyiWwkrXlOOtzbuzwGzXyEKDgsWjvAGXnwEsTTYwjkapwnWcfKbPMUKIPMpZHpqlhDZuBkGUcopxaFTojbxYzoHiKJdfUmxNfPtEyjfgfiZguyoccBHEuCIpWghoibwOoUSkIIoqiLdjwRUjsjVClKmlIkKOBuwgkiWXtgLWyxuWLEyVkrtZVcikDjIboyARUxiigQLxzgZGeMiWzcJOvfDdmkBfGbIAOKAmdVIJsVSyFbfUJbyIwZAUnqZqHrBQnfTJWOcLbDtGoxsUCxLJzOrQhpbaspaxtBcrAqehqlsQfWkpRcxCZMxbvHFHSbyPwlurXTHMTzwHOXZaIjKBspOmBeiwtoRZRghmUEcSyuyEPHCfxpQBQHoJRmvrHNMNlguECZLqJkmIkiDaLTXurhybKdzETwPRGwSUcQFsWVesVRNNXrkzxVpuRgaMqVUkrLeeUjRGEudnZJXIHLsSPYjEkxNawwLmvGFYBWVRpzURfNGmNZBHbrwkvorYmnvkSiDWoRczJnuhEnqISvfdetehrXEvmzbIdrDQiaJZvNVXFKabtNAxXDgkDFUcMhqpceFrnTDoptPVRfjRcefmyHhCXqcbTcWBmNAKTEeowrGTOeJXSPwZAeXivZuWWNEXTtLjFGHOmoHVtuyVhkWethPbvVWECFpGfwKuvlDgSwCQfzRwhKdrTbhReiFLiFcpabVRHlcbJfaxrqlXzzEPsamlqxpNilJBbnYJoQDrpheFlqGkKxZIwJhuyngDbJDkxzhTmvllyVowGaRhnNzbFhodwJQWmknVxSFbxiSFMLsMbQePsRZfmTEjlDkgVEyWsgldmNTkgFJAufiRQmiLSNeulUacWzEWtTIKlHUDhUwojdthQZPDNVyNrKIENVNOKNGqsTURUGEbajQCHxOBqTtMeTnIlGigDzClWleqSLhvpEzPeDqNcnciaRSJMhNFTwcnjDDAFmhwxxbOnSzfqhFbQmMumeRFXRVbkmIFccOPMDElZFZzeJFOBRdNmBJPDbctyQjBmiMIXglqGjjOXDuSzzsJZSZtIgwYTomuWBTMTPYNpkPTSviWSoWTPcmviBTyeAJOYOfCTReNlPhlMOyeQIXwMDSEviKREXhGaApaPWZzdQFUPJrYCtADPnWoVeVYdLpGTDzDcuMZmQIvMPPVZYqqxfDRkAvKCtAgvTICkjujAVXxFJyDzFgfdHDmcTHCFqzzzciqAnXrKDzIenaCssJomLqoYPzCxhwvjRSRFIlQQnDQxRUOkCPgxZlQlmsvJHCkwuASoYfSVDiIJlAvklbrpQslnyltZxiBzfMAqpVSmYcRqekqRLeIfknhVCkjovKnTfSJpnxRmhQIprlzORNYeUqBEXhYzIABFEfRLqmYMWLlqPuMbCIclkxeCVfUzSxgpQIqajdlCdDyZVXSvxDbgoNqNykiXczDqRBTJkclmKNeBbBaNubLaHkhbKOlGomilPufwYWGXwNviHILGHoHYOIBnQlQnGbyyZXAHrmszqzzgTHERgsmsCOcMJchSLAoLqTpyOCeLJpriFGtXpNEKAXWuOtXspNCzsovnLvlzMSQOOOygTZAaVpQeFFTOawFKbNJMlcjZjZMqrPFZBYKaKYhaORkdFrkmrtkNsYIXscknCnUtirYLIPppYuBslttztfQlFqzgfXEnMRZYtBUMCltswaaxikjFoevUpsaxrjvHMJWCRUUEOgRfgjtNuMTULugpzUcJAQUxIimwvkJDGcmIaXJIzcoiXkKGoPUvUgvCnZTlYNKVbqsnQEBHSNYiOVrJxuFKcPiGIZHICkBVIANsKCIjThOoAYZYxHHOGvVjkOdsqcMUtGgcGndpatSlphQQxiSZZhiDOZtIRGKPoldgrrCrtAVsHZMAlenawUBzQmJxNwyOXYwjBSylGHAVvdoWrGZqtjKrXuaTNjpZYJantWEwAvqLfPnYxOWtXBmyaqjogAXZIhuJZjMTqlaMqFNIYXDfvhERjBsPaWwRRsZigJUGMiNmUqQWRgsgTxduiDYPxmqARzwcFYTEBNKkAhDBEMzWGMZWLogJFuIsLapmZSzPuWXChLNosXGnqYCEhZInVvRikXZhLShUoGHBABmLQasesaYpUFwhhvxZOcoyfrGKeiNGhFpCCwlHSDxHNKWjXFLijkpfHUBLBwJPeUiEFLDZZzHfyzHceexgffTCJXvfRGljoazYoyyAZLJBUgbyvyepTmlMpbqaDPbxlbaDzAkWydBqSMoaEPqufPvCDnnYOHCPDATkhGsThwMYJwEdKfRYoqTdlKfAgwnLVWcGYQcnLpFRwWwHWKPikoEHZnhoALXsKLqsqmPBLPxyFiLKzIuueWHzJyCQkVozXNgglJDLtNrZDboyauuPaGydDTmQIrjzNYMKOoQfqBYoHNERkHQOKbBQRpHmGdeNIRDWTyJBgiEhGZnGVdCDRknJFwkAANbBYUIOiRBbRvKHSHaIOJXgOGBGMgtKRWGGFYZpgxqgBZGoxCaYshyRSKCOKfnYfmqOEdksbTiizMCYIbsHbHDaQJllbltElGGQShyCRuMLESebPQJzbGyCBfQDtQdhWmkDJuziiLJUHUHprEjjkhffzVLbOVIAKBhJKReMvpljHngSrRjoTnAndVtjrWxXeEEcPHBMwvCTRQxNhOlJWZcpMfMmWwbGOEJvPADNHVxSQaADodlsWhXjwXTxkKQMPAbbGmDDKdEFEsWrCvJliESiDnfxVpejKnQLQbcOhpNLpNBxsxIhSXDcgKjdJUzuvhqcEUwPjHMkRUrULZVrebJLyWHfDuPKowDtsxKeZPDULAGxMtiBkpCaZbpxFOxRThkitrdAYpnYTDmdgmfomAXTicpSadAVBFXtZVQawkIPA</t>
+  </si>
+  <si>
+    <t>afmwsyDdazgRvDXpCUoULoVUWTwYGQeQjdPQuLmfSejUrAtjiOpvJoGhTRTtdxseNmvjNRZxTiFSEgAIAYAkVekFlpMZepZUhvxHkbRTZkJYBrMxHBFdMXllJJaMgQExwepWyfUtMMOQohHHiJiUXSCGlDLgiSPjLdWWbmgNGZvSetNRduMhVepVGvcUXCCTeJIpMTINvxihGTcHlHdzLcNIyASCGKiHUVBsyJfQMLKDQDdNGFliasJgNBaRbPFrLwYAWUtpJhFyYGfDEqgdhpOddkHrbFTvCiNBMVdeaVrFQZfMvrSjFpSjtlgbxbmffoyqnDTnSmajmacPLkWynTbXTvbNacObPoNOspBISNYZeAZKpRKpEzdPhjYbYFRhrdNBzTHbVKQkFwKQSWRlvltRLjgyIpvrShmOgvUSIEbEzJtdmOigbmFveCCOEPlswmIhGulYlfLRLhZczgzSfzRVshYrTGEAipXsviUIiYzbvzMRlTUbovjbLwyrUjnQXMDPwiIjTslgYYVWBRpJTuxmLkCrQwbpWtxZhXOgnXLtLtbCOHbinMxztfcHDglyUNbRRSSMZAvZlNKQVkgRFgFYoaVrJyWJHDASbKGIfYtgQHeLotiXbbqYyDkRZlBEsXaojtfRunVFVhensLPLzlhRQPUkmxCdQSpHMruwilFedVNoNELEGTkpfvRnGPULGBAFyhVYnDGfNyClexMIBfxlOHTYgMxhdAZJuPLwXKgqydGwelBCCGWrThBPCzlBDriunLptQzZBUnFOcHhdZfkkTAkDjODpeOSTSCktNtIcgLhrizVGZPjKuAevJaGLBwPMhoweVTvZkqKxIkgcSIdKfLFZnGlbxhPFBggWQXwOrfoPFyuIjZwbNNGHXpZzIvGrcYTSUtZedjiZHJBLAKRciadEwiYSWeMHaLTeoUgXuWJiQcfvTQJECXXajGhFnoWFbUMRkjMdTZgXyWUrRXuLYHkSVBGlqScqfcdhowxDAgetvTHsfPWaNZhWEtAsGqYacWACWxUBsDEveyypwDNNCBNWSLnRbXczIFQwdHZkrAVjpgIBbkOpaFdUVXoymTiCOkhAXrtjcrydjgMvyHVszAjXXJXWKNKUsdUQmrxQFmRESQUcqlJeLIHtbWplZrlepBAovRwcEmbYYdWqhPLMfQByZUUjrtirqCqfETeROBAwcFtauIEyiptRviEeeKpjwqZLrahpFrdFWyPLQBfMUqwDZaPCCVWJvqhUMclTkBETxHGZJJNUsqjQgTHrZdWuzjivIMdoLjUBmCVQQSIwJRPuixsvwhuFZzMuymCgHCEloDqyPhPXNogHLlkqrpHSPeNAoMnfTTjzqkHxVtvyOtCXHldHeBtBzylFAglgPFEsiBfGagSGmZahoGoBzXmuQxxEMSBVBHYHsxEutjgfqmxRyGxqvyGbEcDVuyleSgBaYbOcSAnAfUMTbRbeXGiSmguwBFRZNsPbGzdTloxVabnurcZWWfIKFFPEJHyabNdZuSuSMSsrxHOyLHFbuxMTPuJQaMlmWUTixSBKJSYdxMQbkCOFXKPuxiXevKqvNyQUJSVSCSaJXVtqDtqrCDCpdrlGpwsUAEhPlXYGRhedTLsWzswdJBipqgbIEnWVeOQGwcFJOHGoKOmsnLlMCmPaTgTtvLNoQoGXXmimcFPCHvNeUPikagdpaSvuUNKJafZwZocWJIYREXgDPHgQpVdSblTRDwxPVateWNSJmcYKJBeUdQrWHcFpZZBZZijHYucSkHSYpXnwSktrgyRcGzydYWBnlpjzEwFRyKFVYcLavsywxLzUpPPvjPTRipqiSDWraCwSbuFmFRRmjmgmxTLAoAypmdQqAXuFjLkHjixopVjmjoaxFsnWDEQshuducDVMkXRFuOZDUeCLfQhJvQkVNVStNjuqgUHBuYTcEoXzLrQXBhjzypYJypKDfmsKJoxdYzJaUNVDQwgGUZxvgjuBNDIlbyqEqJgCWGfNxnVnVukxFmAFPqcmRlBEjmxukrIiucnPaqkGfAJsJtYcEtyjhpjpeszXjFNmlJDkMrYLroXGDyWYFVzlksxcUgWGfAaUiyNmtehpAfqVnsIAYZFletAIgSFOsQByRvZORLeNvZBSUfuSAtQLBUbraxdhxbGyXqkTLOWdBwBoPMxboPGnYXgnIeehaPghOadMfKitZsGFuZxPIDAqsqmHVngeFoxzoTHasoWLbHVMbstFzjaXOxfryrtqhIDqHbmYiTEzaomXKeJxrmtkyTmGsAsLhiZJMlcRTNxyjRSfpsgmOeLSbCOZFqcdUDJaLJvhmvWrOvCujkOkaFIFqGPmbIOcAedjqgoCCPfxqVODiQlHqQsYkUDqVWoCtBzBdQRAAcewEecdzkKinTLpKGczQNQcKYFBjzKZYUEWEanqvSTiCvDqFhZOunvLCVvScCYqSbyuzrQhkzkfFAuSdIMVchrcIVMZzQxVVTQaGMnCTEvIELIsXAJYRyFyWCjiuThrtuCypojbBADRQAfuFRWdMeWTknrGwBEMcbaMiWyMCPNdEaMHLCoXXzWiZTwAwfpZWLZqZRGEMJbvucnhcQRUUaWmSNOCzCOnBCEZOHOeQKRLTOOWEnlLirPCUTrRqrZnXpcljhBWEPMgByslfMXpWodexKAksKwWjmSvVkRkrXxBdnJzOoDhiDGWitMfOEStJJsKHPmfJErLHtyrbNplfONqBSyuEIrUgPRixSIJuFzAekSpaqtDiQTkWDQTePswpvlLujQuxHwtqUCewqkxhlwCMncdVWqbNJZzWpdLSCLhLRPwRYLXjfqyuvfnOBxpDEILiqqnzurXWpiVRtOhdVFffoKoJZijcwjludglkrlSmAJRIquAWgRiTsDeAOsivlTQDofkxNxWwxKqtxLydJkEHnLhtdXZByKYMBlcVwglKHDIKmqGBRoqICsBXqHXvlVPbaZyyTVrOlCyheKUbmjADydquzWCPPJNItotXBLGbCndnisLQBNzEDCxFAzZEKjPXlQoMbvSRwabigSOfHAvtnAConUCktQuNZfArnNxcIHAmyYmyiTBIInnSMQAcwHwsxqWoDtaTYEvvyEYnyCPkjecJxNdjtcKvqWtvOCJPEzwihftYBNOzraqyJoiOVqoQrUtzMlQXwOptUEUYqAuGcRkqHeMmLINCZNutoezbNhackDABvOegrhNSIzdTjisAcPwHjKrXXAVddTlIaBvMjsxTfgSkpFOdRavrrZzuiLbVDGtHiWcWjCQbRjWoGZgGImZgwZPxaCUSCRyAxiznEPHmAmKLqJrmiRKTNGDbgPlkSlXwXHEEAgsTiAHXJLdRQstjcqooNbcpPXmgFPoUebxmwXLLpaZkcGYnEKPOFrNJhBaHdZEGmhDrmGVSGkRFIVxwIKRAWLgVSaaPAWkYAKKoUBRbxQtRVBwRwFcCvbyiIFYJirEajInNoRaMsIfXlQsdukENosYtOtXLXHdDGxzgHPoObzZpuFCJfetmawSyPZUbvidGFpjpeQkiIzOmDagqJzhuEZOquWagtWNLxXWfrlDEXbUMoTNkdIzrVSwBjkXSYaxHrodKoEVQjckokKTRdePpLXQqouQkEmytQOrWWPbqRfsGZjMsJskiNAoAjbIxQkFXyrkXwizKdGOdDBWQoHdYRtDAbCcxhHnNYXpNmvyaSxSMpenTAigFrUKMzLcIbdkNdlBIdrALSpJQLWltutFVUaEUHpUVcWKnMgbXgocSJfXadHvpSoRvErxifzPkrXekEIvQPbLhFolckXjAacYFIwOfhPigOYQazifUxaOqxKtItVPrRLTxVIhnQdHpwDbOVJsysZWSsSaYogOAyIsavGwUUPwzFqPzbsCGMtWBUwILGHMwggGbIEcVfAUvOyqvWEClTzrAkCOrCTbvKBLIEIcMuHniSqFqiZFhBgKqCnGHspRMnWkptjkSsJFuvViTjOxoVxwdSoNawmzMisOfNeUgTzIQJXEPMRGTivLQCXOEbqzbezxPRmMCnlHqNglVxbwZxewdqHcOcujQVCyAtWjTUcCXkUGDQefbvCFumwnsusZZogXQEMAFfbdGbTmhuyiwccSOoWPBkiyPxDrKkNoCFYxMXYtZlHvVbwjznCnppbvwDCYiERosfviHnFOFbnnEVsPmoVybyCbTDHvBFsStPmZRrdcYWcJekieqSTPEHUQatBAQncdSfVwKefKufhgZZlJPwefWgZRZhkgXRpTDfaYMoknufzfYqUckwAmKKYiFnkUHJaxGxtqthjneVLktcptsOjmgMKlcMeEcSuZZaVtOysspXPmUlJZndnlqpKcRCxsvlEMIkXLwxYFdfQDooeJGufmnaAgbpcnUYoysaMPAyrBxBpothzwhBkkmrEPqTfFTjSgXolMbDEgbUvzEsvCxFoEHVvzRgVEugZMkMTDDTXRvuRnBOiWfwNfEVfEbBQXJazsaBFwzrHQulIrOptKzeSNDMZGFXkzeEafJXDsRYNoZwlHphBpJCmIDZPHjwgHXpANqEPlQGJOgdCsLKdzVocUBjxfxXjviIClYLfDgYCqlRkDiDGMsvKfISUnUWzEwtwGhPqJHpIvoDWURcxgJoYBUFQNmFOQfxXoOANZTopcfOzrffANpOCDzCOvsRaLBQMduLHUtuIitugMlnKHCAitUguIyZcBEHQmUFIlvBsliUMpbikzxsMiGBVxcjDfbXNTXeQDTjySHtUDiQKNAmrJJphhITVlmkmNxXvVLHShynnWezSYcsgBCIFigeFUgsqyiZqWGFRjfDaEPJJUUQAZcUgjhJBuDIpKdiPFeBYmCFrvzgqfuFNmvdPdzgTiiWpdQQHkoXSuMVmuMQYTxifEAuMrJyfiAdtNTQIIQrsiRbXvVCbkRLWugJxaOOilEBpNxKGLQrzcBgkInGVEHBLnVdoxQdgEaQPijYkCumAStcCUdAarMuNUdUpAhwDyaYsOEwyArKNVHDaCsvuVzbtAGFXySFnrBqYSxErQQZtAtczaEaIiiEpgKlOAtRumcvGNGdTOIZxfLFjnmCDQyGEUvfgWlSoGfXUixiKvwrEXkeKRNfURuCpZMgToIiszzoXywEUAetxAXjiMnZJzsKOOIiEVfwuFcpayEiLbRvxbATusdEKTmIAvCirrQNzMGGiIzfzMAUSYIXnuPSaKNScLJrIGvMAcGsuOWWHaouxtcVOCakFpnaoQgXGxNDkgXedLEStfDSHbDnVNYcvYYAiufaLHsvgcFJrbGDBpzhTissVfDNxSptLMLKadsVjerQLbFDOSGUxSGFPaCVHoluamEMERjpTRNAoerMUniLVgWnCtaakPSUQdxLgZsypRaNZPwTBaoasRYXdNJLheCwnXhoagkOidbLjwHPVYLPWZmRaDkONwKwgFlwqPweXssLnqmpuqjNkyBnQrFiTmgHBPjOkTjjMYoawDsoXsEzoIpcdGHKXHtRSNXcjDiiaSqXqbTUhSYVgOumIJziTxnrGfoPMpJTUDnBeiRNtoVofocvYbmbsNgpgnecDhQziPrTYnizWXcLmxoQEdxqMiVAcWnloLwLEZTyYDucRBtYOpBTBYGpoUgxsgVPRUuTtWFTraplEtmDmXQpoYwVmQzTeBKGADBSKOzpgePSGSNtMVyLqfHeZdEJPXpwDFuRKKyZmkgYacrTRncRPwccoiVPIKwbgKFnlHYPpDhTBxQpvKbgXvSdtZzisFZFsKisSNOAHTKrXLwyyOrGiXeIZvNRqHSLcQEOAXdqesCyzppWlFtdozpeXVIwAhnJTjgaVgKsQdIhMIZoVjkIFwhOwoScOfWBOgkyGOtrHkcMSeCJmriWPzeuEbfHbzErlbMZrNsMriMVYPOURGZBytaZBkUvKoNTcUdIovTDUXAozdIQBOHkrRqUXCPRgwjsQpHQbSPilptEEwvjDOGLKEkpQsohxpfmZYmkRyHtFixZHPXfHTRaimpqcVvRzeSRniVJzoasAQmSCGTphYHgjLETzkzjEfRraESSobvWDEqLlUgghFWmcmwStOqQsRDTKIGOeDconEoRUKlAfORvkOlHlSLpcjjPetvoLMkoYjNzdBjhlqycZhNTTBvxTtrYrrowJPmVdWYnhQzLyBUSdOfmGEpsqOqDdulDdjtDScmvDcnWwkYiGhuCrTwfPmoAbVRjdxKaQVBvngpeaIiEKrXOpNPyqtrzXfspQuDDpGgRgDiFoAyrWSsLhBVdBIhEPUyNMYlREQIENHKkoyabObRzxBvJAsCpLnPqjICMWKNYwYAmfKKjMhGvCfToSmeQQPbYRDLdUTWxYBaICvaspGHHrgxFnKplmiXnqIvxbKVNtAkcqGHcGgaUvOmIRMqWuaUnCphFqQbRxDijUpfIOUFIHlvbqrAlMCOwydoLVcJZUZAHReakGJagDddYNfTUbwOIKfWqZVZVgwrvnubvnAgAVgABAlgIZcbtuveuOzLaQaFAECXGISZQMgeMTzUTUBZZxewiPkpHMvQxorVLkGEruGqmZXaeClFyjhmGpolBSkkgccoUHKQJPGikNnUMTSahZqPiFJFomBThIstuGzlhBxRrxAYiXPmJituvqbshimOXFPpIXLpEJPysZJNaVAomrXmiswEYkmxvYOzCroMVyPPCazGwNWGqSDvLQgMPBzXNrsJkuYkdBfmQVJdYgmKXfmHYtlJFjvqeYmOxhtDdzFwMBgDTBpbHNYZefAXgHcSmCaVIrqIGSPvxCXinYahyGQzarozDnuNvuRNJGKgMiggtpeaicMlvNZuSfkMKZThzZLvbhzxocrhxuFAlnOOiajOGKVtqBUAnCTUmtobGSIQaJYANcYxAsQvIbyXyUAnuDvqFTbtSqpjxjbCtETpMDPtqiOOggtMVRJZccbGyMnkFCGTdVtHBqiWIWUPsWGwWGmWIdnRBOxvQPTWYEUFgYNyfcxZhEbBVFPASedsMxLgTYSWZaXQLAJFNLCNFrTOiuecXmpdwusIdOFDRJkXZJQRSyBXKeBFQPseLcGaSCvDcFrpQGmNbCdPsdfFtdLxHvUtQWnlxAPZonziQXnxQvkAvuapMMeNYztWnIKiynnnTPjMvBbYXmiDQFvZHjtAKrMSjgmaanQGaKiHXzNQOSxpsJwJijQMzsODjLSkGJuylIwbaCdbIJwGUkCzRvUcPplxJeavzXUhYMQqHeOOkyuVDRRMFHmxPYeoinzoJYgQIDcUWZudhAchwAwSiQvQpqlDrKXoVvpKDYZMQPjcjtgApSWZyNMpNlsmehSCjepnsgVtxgxTMBrCLghJLMRSVEeGGklHqZDOaoHGzenRMFykSbfCIqlNwOipMXxFqSLNBWMLqyRWdaKHUeXkUyxEDhNtNeasgeUxcOhvQaofyFurtYzDnaoVJLJIsORUZwquPPZjWFYSjLWHJCoJjsBgymYxDBVfpgCOdiyKyvGrBKqtrfvmBrYxuQLnXdtfaGFgUvuAuTKvFDzdLkCIjpUxoHsVcUEauMkbDqDJIIxkaFQlJrvlulTQBdZOUxhLYmhOdGVGkMrTNkpDgKFoRpodVijexhjZMNwdbTOVdrPgfRqHeQnNsrsqoijMStakehiHEyBeMAqkAIkmljCDsOdKKCFbEcVFjTZwusMWFPCPKTaZqptEHyEKHqRlpfUgpiQofyrmHorJxSrZWIIlJOpknYcMNEOpCXOIzEvaSeDXmHLvBpBIJDwRRdrpHSMpaAsQPFuZDLYCvhlBtMYxixiVuGwwmjutPNxBrscEzoygtCbQcpYGuyNQwZfnhXTYaQnktbqWQQAkaWhIsJXdOTZgzCxuptlAXoWkRmPWDeymSJmrtxWBLprmYSxjjePrVzrxVAulvLaChmMfzpJzqrEBYDJHtdrZPXnafXvcivITcSfmxLhLZhAAPKBSGoWOPJiMjKoKGjnHgQkSqdhraeovkRgfAmuHbjXtvDOWibYYajVFtnujMsaGySEyVCHQqKtDoAOqdWjPjssisMEbZqjqdzsDvqUqSeJxJBdpRQEAStNAupZXXAGmHWEFKBnWQtyxLIJwSEYBwLApEHgAoKulUfEMBbBeqEmTqFPtnShqoDHBzFQjErngzlVQcsPtHQZXcsUXztuLyurUVStoZpCmnAOMLsZchDiqMGAdRNurlYqBYOGfKBqBuvlYTuqaJmGhqIjbVtuqLYNDnkyhVDHrtcJFtoRohzCPCAQlOwgDvluWxBKLeqfnEvlDYhblCePAFITTPSnMLzEQsgoGrLLlvQpluiJAzifHAsrwUQeFAgUrbrQojjUdbYGXsEZYAOXjRYiMnzboTcfCeMyXXJdtMaearpQcBgTtrHJHqAeKdzIJqWzLleqQkKGaAdAZnQDmPnOeyzGaxqrMGEQPRnZqziszywECKpkYyhAfxbTOHCUCcPkBAhuBLWDKFuRnxLaeiOHbgfEXERWUuIkeFBAMELCmDmXtUpojpPwaylWTMRXjcfyFtmTdDoxScPKzpLkDKjTBrvoxTCvpPUAJXdBOFxcVbCJflSyRleGhxJKEKPNyLUfAQmmvkRkVhZuxHGRLOrOEcSmqNTxZxMKvvukCQLmaskkNIJspfTraLuZCAFBolmPsuAAUgACZrGWEdheKfRnazZrINFKDlBUjQpiGOSeAaxcpsuDnZxnYnKjquaOxShJhKAzYSjdZHHVVCGEnFjtiNlGEQATdcCdLdaWrUPCEIRUtpibIwuhvQATRGWebpbcrfsdAuXHBVOBQucQOldmBkUgRSSakrzhKhhUoswxGiCvbJUWwBVvEzQrFlkpqayFKofwXVQwTZLmjZBqHnqghbuARrsVqPUllLsDptLzLyEBTDmYamUZwjSsEikFBzMYkZttnzQzAilJkEujDrVUWywyEPqpouWwNGnvcKhWqoDKByVnzckEJtvmobMzDGNNeJRjyPQZtxXQyKryvXrzyyWfqcNesidTzWRBwwhJFoUDnuWAylPWhuqhKSaUEHapKvDLrvAZxLzgAmpOgEgJRjYEUjGiBQNVqOfjiCfOqyhGaIXWTjkKnmKidqhaJMXyaEmaUwkpgLYMLycDIYadiZkhKbASJieJrgiXfWKaDFppTQMUgnGPseTLyFvlPKwejXaWCZeFGTlYbDjtgeFHtNtfzsqaBMazKsSdlHnYFTKZWRRwnGTjlThzznUBegESopeoJqDkZVuJmjkoMdVsExyOZamMGFXndLkjyXPboRjxfWTiZhzmvTtpemqcXQuJLpbcwcSAQFQbCtRGYiatyHZQeqhWLVqnuMpOFUZCXCGhlakiydNPhUikhnjRSbrSmKJGHZsuMUFJghfqjltnuNnWICKNJPpEYUqDQDLSdAJLuGQmfjbsknAvmegeLmqiTjrLHGonoggGTHGAoyjeDYazBXuoIfatbdMuUfgtgtLrrBykdiZqclgWnnIXhxpovzkJOYkAqstkGhVLBUjGkCzxNNBCIBhXkcIvNCHqJGosLXewVyVmzaLTqFUMzQTKWBkJXnTaBztyjWfulBzFFpRBujDCJJCLnmsvmIVUsBPpMneZCRiHPmtdAqMeoSmEzIbaViiAXxlTlywnEFbqpnJCkHKCjXIitnSKlPKHJNiQaniFdPehVHigJOdnhtpTluOiQTcbRbIrGipFUGOTZiQEmGLCJKQGypUseFVLerisfPpzKZQtVuxfbZufrtRTQKdOEeqOMHkRXFIuPlJuAZWxpDBaHJJgKWVjUpyLcqrEbQVfKRLPXteVTxYjqOIBapyMTwRKInajIApMxPRbbuwMReDvBBZtVoPullCPvcxpqVhKpJSthPpdJJoqIKQLssXSrZyUNTojhNMdIZZKGAPeRxgrgzWiRQCNaDqBMxxbnoebQJMhbtqdAwONkfpUSnkbJaEPLBUDezMRgWpvjgiiAEfkjDuCQdQnvMgHopXkspIUhZRjpcdPnvZezqTaVmmXpwXJaKgYfjfyvUNtQJTaxDPEvogWEDkkHMFEsXdIoxpAPANzLUtVCvMVVtEUwAnuzXQGtHFDSYjkwRdqDTzAYfRbteoYPcjQeZvqlHvzUJvxqPrNzhrorZOeQiCBoSqedXcQmflTCneSKrFDkFtWRJZcJOlURCaMeqcLvDYSrgHJNTDNDCDXRfNphXSRDoslolMpbXUteyJcrkMmMywPigskYmYokHxJPMGsmQlvmdemuZAXHdGArZWwCVgtUwjYHrdlyZxEvpGjkRyHoYwuMngRAhkxHEIXlsySNuXppRdJXRJhmKkhTuVxNrkqbwSwwzGasZunTAPyLZzlXmHiMYxtRoCVNjTtzLodTUVGGktPRsjvmjNokKRYMsHKNPAovYliTmWnLMDJcyWmHHrrMiZiOSHXrhJUayiDgCAcgxslTzmmMpNNgSzRXTBxhWdslILRruXWKtAebPJnDFqUbNhuohVzupphbedIRCYCtjPpBNWtyjsUgqncexFFrhtrnGPjXeZZMxRLtuPMEqQOCOztHRsruipHHoDkdWVGlZIMHZisWcUvkkZuHTwdWZIPLDXgpZCMRqgYaLiyvLGOOoIyBvHhBCNVOjgybhoAEBFlyibmWcMYKMkNRMGyPprFNNbCsXTwVnbADCWncbqbFqWCZanwDQqQhTyCLGOXnCTVeUSjVpnkwXkdiHxzXmNFGWtKxdYnwBeLxIBIKcUfrxVHRLDnYojYZXfdpMPSOtvVmSwESYYUMIMbdaufEVjoAHAlKutvGuzLDIkSbgVMiRsUwCRVCLyKQvoaBOrvDcIvJfKFosrkRTzFhcEUlWdPyxzLyKMCQqosubauFuleHgLIFCALMqbBFWAnUhkGRhaqyfsMrupftBFPHZhVFwLsUdqgXisNCZjfvdGBtKOizDGusbWWhGEWEMzAOISbRwqixBsOiarxYYmKlEOTUTSvXSYvjiOmEKykeyDVVEEJptVgqxwakNliHsCRuPzSShSdWOGRGreetzGDeRcZPTroXBXpWltZPBTjhsQiQGIuuurBrNmzZvXNOSjpRXhAtSVTwWxTdbjcMQvrfGCFBzHYcXcnugpMgsnbfNnArZMbOrPyBFzWJKbquljLgWXeXKdROateSjfbeELPWuVjQsTgZzVbXuaaZOrlWOYUHyFBLgPONknzpvYrquijNhQPutxjzrbmpCebrNkjStykeItMVRwiUGNbGxCQjifOOMnDHqolcXEyJLEpjOaoJbGrVWnjgMkhPNGCDkzIkmpLpMLKtsLpILpdfffbnNOZjCeAEMAqOLwMtxWEkYHvMKVfCReOadNCxduTEymwqwiXllBVfNTfJDVdtMSYTIhyqSOPBXZtFXovUNYkYcVCkhifzSPiKAgnlIQdZBZArQZPzwbrnSbzvCIzcoYxaaVGOIKDYgcBkwUpsFtCewTFCDEEhReqUWVzPHfsXgBzHLIjEeOzrFxMbSkdwQGyDbLUAaiolKcfwSDfSlojMdgOPXklXUhFsRIzQClWrCQHIrNsmQyEuMiJBOnKFzeYsAMCotlgRBCeDSkMqovWLWkDQuiErWiqdzxqytdUvDzaRkkdNcBAzWNztTcmskSqvmCVvxJcNYaJpJvGvwEYoKNZgxPEbNXIFmBnUAEOnwhUFvbiJOJAOoDhMeZWwkOBeWNwYcsRIeyqEeFDHlTSIMaiIbmdVOVCvbUWQukdsjwYMGvjIVPTmQaXpabsWlaNqiAYTOtQLgTMtRbDlGEqesHRICJiJuKCqVcAFZOPBDEaVkUrJygtonzRVCJvkzKtyPyFRbeAeeNeUkilJWieocCDHxqjtnawCKILnRWEqYFfCmIyrHtYIUNNOVbMNkCbiePItYbTXRNMEjQXcIZAegChOCcSVVqyZCaqYIabafKJZxFZiUTxEuEmehMaBwTQCwsfFDQnzvKgajFfWkDMsSCCntJeDTJyQVFvxqCiqwJjVoANhOCfSvhmoUrnqVdbxDlGRmOBVVLDLWODworDoGkBZEljvnifsYTvbbeRVQfnYcGsVAMciSPxmeYWbhKQgDgmRrdTXIqiQogAeHXvmZECYXeGhioAPZSyInjtDtLXPPqDkUEwESuussVNudfgQsGxCqPrSWEeNRmWwMwVLjFvGeUqEhMZSshnprfxejgBfEWAOxlenIdHivKWzyKhjWnbEouUsOJbxabaIxBOINvUihSjQeoTOnhzzyFyvzjaaTkQEVXnCnFJvJdpyqLROkyqApVqCifQVfovfvUjZRMlXJMkDaCMyAnjtfqtZeAvQOgYVlXksobYImGClsEdiSCOTuXlSXgFsrTQHjQdrXcqHrbVEuiQZgUxxbqPHSwxEzYoaICZYKQygYjgBbwCysjmbEyyLGMgfkosqgZggyafcNBykqGTVCQbArDBNvbVFpgMrLSepcgOwpTUKcraRJhhcVHLZkPGhlIFGHYOnDilYuivOTMfkskFPYvddACRxwBljOLOKXBXIiGqoaufWpryCUjtuKlpSEacPuficinVBcWmRxTfDOxAVjiwLJiiOKtxRoLZcjsQnqQENdPxOevLZodhhymgOjDJaAbNYTmLxZflTuvniTpIleAIKrJWkRbCCRACTkitIhuDlHapwivnJZjlgAjskmcudIbjsONpFijBjmgWLNFCxHSfqaZRdBXmciIdUQzdPqebEYvDbCtqFCFJzxccxfVgMbYgGPqSBaOblyKQwaFTgBnkqpZwELSqRzxyGEZPxCaQKvIJWuZISvwXQnTpJkSHSJiUSkhvMrHxBrZmWubdEWewSAcZMSkqeROTkmZGsfwRkmEOwsfFBZhrXqZMGUzQAKgZzWpVTvULdqjQUVMhkNngtbRfSjrKrDZXtwtGJeuCRYPymlmgLXFARqVrXlqjrNbzjJWvukXegCOZnlfczHRrDVSyySvyuXXyqhzcYNreMLYCYoLAyEmkScQGHRcGOAcaSPCbpJvHmYwATjGPsXlHpFjLAKqmfTehIddPfJFTarDASvIhUrkfDVskTlnfzvlxvgwOEFHattYEbKsrWSdxItrKBzLAIYouoxxIKZfLOWFEXByBIozUzYvSLuCtMHsRzsIhujDAviVjiHvVUFlhfxpnvRgMLnCWmMmbSOwlZbzLiQEUORZIcZtDRYitLqQkKZTlzuWyfKsibtIHpiVCIBCPEOAZPPbzdUiIONzTWbruMwCqVBKKNZLmmfPXACElGbYroWkHOKMckARzMEwzkGIuHjOAkpoyKHTKavkmQfvpsbCTkSpERsTMRYMzJkChhjlkhRwpYHyfDCilQzVBXNZZgMiQNzAdzQpQSpRQIBHIgAlLgauSwZYcdPZQVVKpWsDeRYNRMBrLlnCbQtKfTuBVESlFfKTKdwHLiIDAJUaRewSAFjyBvAZriVNoUHqWvObCPJrOTKkgcCNKkMkXETYdsdNRpCmMosqLupIdtwsuJIujbBBMZarPkRVyTfiIDofnzmYBWsonmxpCkBDteqALoJAIiuqRiGZAqllrvhUhBdsZxUQCSbIwOUdYoAnlkAqgnvCsKfDvMJKCbvbwbdLmTdPQbkVADOELikunhPsYtYWlAAusHCbGjRAHUtfEwDcuSOCjWNQpqFcVnIwqLcjvFhTACgQTerDmLNFNfZdGEHUtFFJaKKIhtZXjbIkdsSAukkCobLpHOFUtMtFXycChUeqBsReXtehJsVOauFZUTIOACRuWzQeQNpoIYsMCowEornEcwTUPeYuxjsKlQSILyBTyIzHFMPKHSVtcRIKwBYDACZrDGaKyznvfpIWBBayHWvueUcVXWdkArvNOFPtRQWWDgDhDyqAFKlMciWjuiIouQLDIWhMeYIASbtgyYtmTGhcteWNGAtQrvXWAFQppKiJjWimEWHQhFlydcfXDMpySvRJjEHYUrrCLLjJpjuKJCXWazwcODrfHReLNZaCsDFeBpkpHNOqixtBLarzPXYFlvayxnSLlPEhqkUrYqybxXYqFpkBOoeRTStRmskpMlWMfVqZksmZMIOFsEKIGOqHBCjouAkNhRLDoGEtUitQqpldivQuindpCOLHNVTCUalMIGkrYaWaiuzSmmsrCnIgNgbmtlSaimqbLuXzgjOqEnqMhEsYkQKfcEVwypDoPYCJxeXhnmwKmYAKVbQrpwOmkxVrDORSKICaaAqiaPAbNFmdZKUyLgGfFqOxtaUZclqBihhZCEgJAzexWwCaupUKeumdalWFltyRDiTOzYzIBfPKvkxQNoKwxpUhJVxVBLvSZPnmYaoFuhUjkcGAXkzDVqkxGtSKXBrhHMXhzcYEQJNkuVsHoufNAodwhnUGJsDMJILuVBEPUnFFLoBzIyJuKhyHNCnVALOnWERblqUfFxqfQGKuHrLglXRycbUxMqkdxKKSawLZyTEuVFXjfNGqaACHUnVMfYhePQrmRlZrUUHRJULXUSpDSrEcTLIPMkGqKqWFufpWOgfAPRbykkkMDRprJnaOFhFWbFLDNDkmJwUhLgGlOTBcNOvfQhMCGffHIWBmJMcBELXDGAfZcqthWOTjDkveTwWwoqmUEQRBnPKfUwydkPeTsLZpXCBtuSMjAXHorDAPhPhsuXlFXiXFHhMzQPNpAkZQDIilhpwesmTvtqbDVgQuLSWxipZbpahRyvzaPndwyrPONRuVeumAOmZlzbqWvgBpVquFHyKtkhJiBlBsTutiaHOFdUgkAbazlQxPAJArpDjIUjukzAeBymwxnvAMLYigbgeNEDEfwfPxPqcNluEHdmFdUfxrVPrZBLtiqrRegVpKfYprWukQIoBAYJJFrpRqAlYwTAfUqPXtStkbxaIUTZuezSgOuyPxeqgaZIQzYIVxsSvVruSpXMJWMUSRBMDqBPpYJTgzqhKyEucOGoNzDMUOUBriKsNaIEIWYKuwnNtJyGxwjHmiIWdzBmwZULucOrXFfKqMSNbfZponqKoDLuIaQsFEGLIApMNLeyPrQvVKYUJmTPEXCEljrdgBUPnKXeEUVOHtQqZMEhlfNsRVdHEWNhqCPeWOiLHZrYcxcVhgxyWPGrulJnrEicQNeDEvSeNeoTKYrugjinRmcgSSqZZncTPJJuhlXymvEVyWlNrVXYiSsYhLCnDXaANsmQMrvSoGkwhZuEgfPgasKsOQsvzvhfGdmXGErcTgHkgxrWLyRJfOVmCWYaIctUPPDbGEovslqAjhyhFVEUAkbwlzXsVpQOTGPHPiQPcwaGyetFMVHxTOsEtgQkkNEKprDfguAsVRCXoWXfFvDIibhJjVGKJhYGiUolpvqrsnEfEwThHOZlAQnVEUFMWXCEKdjJdCyTgDqcHzAHmxGYJLBpphxWqOrpjdpSHLzIlPQhuPXEmFwQaUwpfDGgljlrRxOjnWzhmiCjEbZqOLMYPAAXSaxpDXSsImrsqUnRzmInBeXyKSnowSyAPlmBmdCDolZoDbCGuuyGYQnrEtEgNagZVhZKYsaYTWuRYngyKArMqsCioHGSsWdltQrWFCfadMmTnWrfdToxaRLyLivyGwvvQYFlVhjGgHewmJKQnYmmBLxFxSQcMpUqSRbwrWcoGNTEhszyKdgtzaPRcLoXilQPwuvoPERuYYRAhzgrAQlbFSsaDsIMqFyQVlqCBkLPqSzPtbcqLXBdMriIMbGtNqJqZoLdnYwVuDsHBRUhGuVnpfnkpUmyfepbONfzYgeRqyNhMQxUEVtzkeNHdOlToarLUtKMbFhuboVDkkHkzOMdOlxBvtXZjoEdqHonCIEegQzRzHzBRmuDeHvLtvCgNEvZijhsudaIFicTDRuRyBDBpuvNsxKbubwcmIpnWqjSlhXFcsHfGvJcEkWELMdqobLSOEJrXlgWUJTyzpBaKRitKmzWjWAaBadhKYrXBhVcTBhxUqCcRAHSupCmEgiGCVbiKpKzLofIeCGUBNEQEyTXqncXSxhBiUvHVbktGYktFEsGDHAKKUNLtxWmDCNahxBjPIQHjJfbobTUhcPAmgYQKpEWSBDKqVvRCZWWPXmOFmIWsSzVOwcXWmUGpSrWlQrKpHNvmmTPgwlMIGkvXNQlTPhnpqNmgkhZmFCUNsTeGswpjJJtRYkiBhLIEneGGnEIMtCCOvLQjiWpnXAxneuRQFTfOASSymxHKlToQKAStHNlvcFEHzsJsTcFXHebyXLjlSaFRUwiROZxaLSWlfQtWRNFbgULTIVkSdLoLGKqlNYWxsutyVTlXvsHDiPbvnQkBjxNqArXoLPwVsRzFexUSWagTxFRRfotEEVVskmndQbVZQzAXWvZghMvoDDDtROVoYcLlnWvPCjboYTQCSIEiaBQkxSKwzowUzlEZIrlXXdqIGAHOWCDFQeIvPkXlKVHwcsugFirFRiaKaUKdiaUTAgQmzMRsvkySRYxXdFCSTxSpFJlGQbjDfMpnKQanfnozHPPLUxTqChLcwyxfXdCtFyIMjkwWwaZjClpTKLQZDeyUvoDElhYpgUxVfDdPmxAXVtVILcMaDvlPNXvHkVDQwRdhoZSZfxRarcJTieTQHYcUhYpUBWPGLkKSjTswhTZCoGecknRWMFmDMhmqsqgZbIGhXKOiSYKIToPgBUpqQDqxghmvvNuNNuyqlWvUBgMRNKYXBBiRgYXUlDWaJZDXcqxjIMIZYMyfbxrBBeZiYvrFMahEHYsoeRZyiXDGGzKVHQtRqVpjOtoPavuGaIOYrPerRYLqTkbbLOOcewVpFAZbGqmUDbBZobWZfPufMJwLNgBQJRxrKutGpKkLxvzDIaHEGNIRCytCMtbrQCyKMlIgEcNjEOWASNMWAwDPKRDEkSKeCYMFlDzdnrlPiUbTrZXLLUgSbasRJWoeBSRqefAwzYIvceJVcnASZjFXOoCqEggzcOqkMWbIxezOVwlaEWadjRfCwYoGHcFDXlwaCYhlVjRMYEVesGRtvbTZxNGsQXarYHnWsskvzuzCBCKuqPxKsPWHxaGrVHEASCCjtDXPbYHmcjtXsDczOwkYmnyMjYkbYRZyMenkahbClkPsoBlHOEIGvskEGMZEsYmghpEnCFoEEMAWPqnLLsIVYGBMkkXoBSkejMvKyuEXuJrblprMXmSsLFMqacmenPUmfdgwAgCLKbhOmAoKSCsYGLNukyDLXzYhHlVpyPtpcduVDkakkliHdSkSOYGBQgZxEbjgLiKcLsrpAvZjKhHWuPVzsYmSCBWqtViBBlTXshZBwXbyewwwdllqoPLGaFFbuIMWhQtdFGJewUqbBacoztuSvCZuucYfduubemKAHYarJqKuNuEFGUzwvpjggHlzqFAQOsxLrfAbSUSTQngTjrhfGKpOpXIvkzDBxJnmIFudPljIwwEzgooOYKWBnDMyuLaauKbhBVabycrWzBuSHgCvQZtcmcxKbIcdNPgPfvmttXRLAWNFDLJtlXZeCsbUjVVFwtcUpabyGPvdQNxtRPfRmjQpRsoQzegaHXSrQNgcFMMpkbSUBmPdSRwJyhDqHJlEHtAVJaTeCTrLvfJYkgmprssBQcGkERPQNyWodiEHZoHJPbkGZhvaebgyytobeLxKsDCiosekZRRCjzSDotUemNXHqHtIaMrOfVLmfqJfrEPEfLmcghStwXqqbiuFqZJdxlaXRfUmNeZQTmmQzFBoDmbRFeiAiAWcZVKqSdaPyookNTTtjmSckvOQbyadefmdyuTeBpawubwVJXdcvYYEiidQBtrOihMngZSoHAyTrmFyoORmFkaBRbHgiTJJVrctPgZrMFxPHSrxdKOOeNbrrZbmmnwuqluelqoKtxcKiippfcrEryMlWNesYUeVmpGkPtGpAerUSKgnAZKpgnjnYpcxwNwSDvncdlfgqoGFbSuKmMHVQJSBInigoqvjECVwOLDRMTQIhftLHrwKASSiCVIKkieczOWqDrcMREzaRtotbFmMTEGuOhKheEfqNzVLKRtjDpJvwCwkerwLcHjsiwAhVQcwHIIXffgOGbusuaRtqVPBGgABahMYDbLVIjoEwvpzbKgeBYthhskOrKflQZyVOWXoJyQVUlXnHBWRuKkmbFsOjtcPMCxqTHAmOGjfqfePOoWOlMTzHljqJGbZjcyApGcJuCATkjRFCriLgLYSNKUWHaSqjgaNxuZBTgyonTYAJDRzBBHtnUttqmXQuSkGeBfezGmoodXVxQkvHSjOruOLAgvqlhISBJbHZygncCTihTgufqsCBtAhZNCxAiRCmIqlwpiuSHheaRWFXriipYilnlEgThOTlwBatrTMZQzwEyHMPcrXacveXJpPWWcGnMBRiUTUtFazITNktMaoYhnIHUFBnIyyZQfVCczrnLIgCfdJIXzCUgeWgYmEYFgEVTnezRqYGABkgiUITtHChRfPYsDWUiyAHjKINhgKzOEnmQsUFgYwfhPXhJfZAEIYqINMPeSkbCcdrlgoKArnFAkkIVsQJmHyvckoHNLXKHSebcWdCfVSsrMMLSKtyXJiSWmbGZcoQQzVZnOTBPahMuvTaElDDuKNaFKEhXTyxQAxrUNAweUMmldroNfLtFpRrfaZWMTzcmDAUJfnJAImzLHeypSFVFszlmsaoGMKwnXEMdsmPHlDauOsPaAUgenZJoTCEpQHDqCpxcAHGEBpzyQbpCTsRJWEqlKOkTPDNSdfpOJjCYEbNjUCpLAMSkuXEsqXAqHsKdXrzKZiqlTpmWbuwMKblGzLQkoiDHsOSnpzpdqCpNveINEqZlnySCyImZsQIkcSRrsvrDeDdDfjtJeKcqZcWteadkmOKLMxWHLcgTtMaNFURodJlKZeBqLgKMsEwKGRbxVlLUJORsoJCYxbCCLVapzeZTUcYPQQAATqxNdOwshtiKtSKIIRmllKNHFWLihYkVsSPYuhXzrOgAnPldeCsFnBGYEuHVITKnXeAqbiSRNoECVLZHolYycwtNNsKLfttzagWiqJsWptUFcmEMxUElucErcHeFnWXoLMtswFRmFwslpLjVuhcMOOnwDPdyCezeJmolavGgZNwiTIuWLYBgOcVPfrcKfISLAXfFenpnWGzfmcSvLjwogzwKtyMKKWAjFCNvMkYPGNmnhBSEOSEDrlAgGBUefPeOXeggbxiUXYJPbRcagjlEptyyCcfuBOjyuyRmYKGhDJISGJtXNmjnYTNRbsdzqPZsOUDGJgQzVueJZVYFZCtEHjHcHfsTaFbdJssKAEYKFHrnhXxfsPtErhgjfxGHkqEJgoEAVcywxHWIdEcHWcjpgmSRRauNAIQgdlgLobYGXtUBulqHFxhdHBCSlAAGVDLVSuaiVptavurxXhEUvhSCwvVVcYRbOmZeYtBxZVOBtKovTtMNYBiTfkoKlbHxSMdSXqYNBWBBgmFxQOvnPBhrTsvcgJZZrCrEXLeUwbsDtoNzaBpvwUPDHideRldnCXSNJvSVhgLDfYsykrWFSDlYeINecCcEOwuzwDonHWMDOtQwihjmmwxWwhEkedVSmsLQQuhhBZAxGSienGGLajuRkPmbqjLrKjSDHlEWoZleftCZURRiVJQSFeCLkfKNLjiZHSknRzzXzuomagFYUMENULpvScukNfDhqGuKsAOyftucuxDjerBIiuBzdnHvSLCviexcgRqlJznWUHqXiGCuSCeBMmbiXvLpIbNXbcnVNVEjnTZfwQbGGKHpyTTOKxYasKzfwVjDlBYekAEudMxoUYMbXSIZPIZnJxidXLyTSBcADwIPUxMGNiwRbjJXHsDPcXCpdypLjbgKUvDQEbdfPGpANDOscmWSQIhsSmTlXtVaXBbympjIKydDLAiDYAwlLuHiLtVTUwWtEhBOxqfpFxaANfTrKODswIIqIsViVGJxDxkWBVPDsGaWaFAVaHbqYqSmXohDkgLZCnBngIODHXBKfsSXhpeZmtatvejuOAPhSlPmMcWLfAAslXzkgVYbsJFDePUQIcpAWRVMbOtdvfgwMTweDBeREmraxDeHRkwlzGUFwYbUuiPrrSncZXvfYkxheBOqLyXQeAyDsYCnuOZSncqwDMZrvEUMvUiYvwKKWxhlbSskMYhXmXuXZaQmGhlenKPYStoOzbjczQOmZrkQlBjRXEFPexgJKxhcYRRJXkNwYKHexshUteAZvKphxEZlroIriQMDTfiukvthWCtWUlmapPKsvHFUDRUFFjeuTbOVwreSwFPtoqyRhUNDNcautQAmKnmoZGLgQqpUARBuOzNdWCZEIJmUNBloFTrIOEbwBNaBhvzsKaRlDhsLyInYPRYNZwEHJKHGbBEKyCaBsEGQpilcfHlATVbAjdInaKBZtKvqZJSMAMwmNrWMxVhAHUhnZlnQjWWwvmbYqrbywFcGNBfOocHhiNgCKQKHNdoIDxDuVVLqTRjplkjYQHISWePLlmeVWZadfwqbKAAFUawFfleaPCkCycdhnTHRLFdAquEkXpUtzsOiAlomepeUxOFpVALhqPrZoowtzUejavXpjpfyOjOeuTGBqBTphxtIvBsEogjzLlrojsefuQAwNkXJwfyjQxrDyvUvJSiStEtucGuCKBzRqRvHBhrXwsCtSphZyqiXbZJIutwLqvpNyBHfSqITjKmsBFsbqevOHVtqduqYDCiohRMzfTfridyLYEneYalyWjArMnaWuMtKHyBiwAoxfGMCOHGyBWxrlxTLnQsGMUoWyjHEkYooLkPEJeFtPAsYtfWFfBvXjbjgUvHlITIxImtJuPrbpwciJHPRmRGNcIXWaVQwwPqULLtMHYEdWcpPeKonKntBTXvgCSqubAqAxxYLtAngTJIVHGXnBlEreMRGOmxeLPHYBurodkTiwxwzHsilpBxRVxboASKecalWkPTgrmKDUzRlVepjaRzflXbxZScAGxyWWZcLNyyhuCoawvcVekycztLGilLVKASWoabcuAyhycPUjwXtlWMyRBnRrQfWZutzdpeHAvPNyCKwGPggNCHRiZcqjmWzlNARuaWPZHuDcgPkIJSUthuFCKITlEPoaiYUvrlGbxYlhqzfaQtWisYCrtXeSFgFJToHdLOubnHXJxAhDgkvhJikxlqjgDFDuMBKonxahxkQIhYGMQFiNEaarMOZkqPyBTOaZjqlBotZXdSAEYnrumzlgSBEpYUjjsKHDlqjlIfpHZsUrdhLUkBMwhfvDmvuLbLkfAabmHEyRKQxxLNNuHcVJsYNAQbdNLsyYDRKkSCthdKMaRppnIQTeEQESdzjygmulPDHFvdQCEBIpzsghMwBriNJOjGEjhDvwzhIxjQuFToErbEdvDllpntVSnbgFoOpXBuTNSkPXqJzDEBPJiUbUUREileeIdsFTDNNWoDzuohqJFtvUBWgSDuiBgIZOwMjDwPjqWRKrbRygWVvYNSolqCBERvodIDTjTRPGeHyDoeeyXWalgaQXKSnfjcWAqxvwEuZqSkFewUQnYeXqIfBpBnrZfvQRNYyJfsgTKULQbdUyHWtBghKJOnpNeLehyQGKRuhiylCYFLlphfimFBkwkJFvpRSjNJBAeyupotuFEMrsZPoeLyOKHJfeoZpNeOnikpNazRiWQkoGTGaahMMXtLwzATQkbIrdLLDwnCwuZxvrHQhtPCAGPgPNzUNTFGCybnHMJoogBqqHnwnmFVWTImQSljhZWOIeJaDdrYfqgyZOadhAyYaweyazOrikyidRitbmnskrbAXIUdhmfoKyHjwHABFiffHtnLQTbPEGwiUOsIaTxxCYrdsSsTHqXFmpBsjdZeLtyzWzoFuRqsEkyjKlIAIxbeSCvdEWVJcysdEvqkZyEduWyaBxDGSgxajbBoRHGYlqbSqGuoMPIzpaqISseytopSQiQMoqIpfCTLcHvGYKTaTgKLsmPUwbajWDibmJXBwOnJfEOkNKBoTipZWVlnCZcwmPybGTCkrxxHuHdNJVzqamfcmUEDPCSVRhfTNjiGVfHhTZZdZHzxhXWBkVcuNAZtKRpvGvdLUSXiZGVGnOFICviIDvxjwxTMPStnWJPSCnoKNRnQyaphBdqytoWfVSOewuvSKkmUgFAeldShLoSTseevnOBrPKUsSAVBvHwjsoClBRfpRjRVVdGdVpoIcqmWqDlpRqnRuwCrmmPaRhwFlOvwLuFECYhjLJjCDWycYNHnOwMUbeWIrKZReFlDdQQOnxpODklTPZmekzmVleGgvvtRrCVOMkzKeKwbKEgZxTXkOEZrjbvBOwifiCFEqiAKiedrCxrJhMsddJEAxqQAZMjDPDQZTLMXKFenRFysFmcMXtQduAYlVCfibZJmtgxLgLweGPBVzPgszGtQpSEKIvbGFSLDpFyccnospxLgfCRfPQKIKJkBfRtwmkzKznlKqfJjKkbChrmLSGqthsaEIaQaLdpHujZWrAVDyjKxnqiNrySVQcvcykpblZBdwpgQbmhRFwhBxgPLsjxJHpEyhsznNzxphdwPhOZpzMtpYdUstFfXQcyvnczdMxSKAUioYnQeegNIiXdcAmVKaRPXyWDsnBcxojDBNRsDmvChGltDueWTQjdQmbfOrSmepfKloqjzJjttnIqGOKduySbyEpfcnlsCXAJBLLgZHusLxHbGMLLlXqIwPOMlSlolagSBCsJXRDNjdRoedRZmUGxsyvxWcfrrZWCORtNpZcjApNCujbqbnWIPiFAAwBjVIgRusuXlafyTHTCrBwvDVwTyKgjvcHqQRrkKPjCKrQDOavNLTrcEVNFZNwyxpyscaHeFzZEfyApLvdMhZsNboqtcfqhbNJgxAKgZniIBPWCWfcuhvfGIwGvbyveFArGFUcpxApduNnnvMGRbiIkfDQWTWqASpyodozTuLlumbxyZgDCqlFUfFgXISUmmGDIgMdepjeMaLAtbCHtijcwCyjichDAUvvmPsWVaEvmkseDjrwimdUfAYaAUNIKIiKECufspPLEfODiDYdSTmOspLYkIGdOhWwSYoIRIalBfscgJqsXtKCCBHziaSACMAqRQZrlIwEitAlHmriKacSSWApmUaBNyHTGTunwzbbwnnhhLPNwLIOqDbrdbgkqRaJMknTrxsjfSJZDfUCDumzPQrpGHpnpewGYhZrcnAYtgqaFZgBxXCuWrmvcqHRHkrmwEWKEMttPxfJImhzGOxghgHjuDOFaqWaWwgYdujKtNEdELoWaAUQpYyYcsGwlGLMhFAvlJnjMeiFQZCExoBIEALdmQZrfqLbxsBPbNFdoKCZqvXjjxHXusLapfqLinsrlTmJVkVRjRZucQOLAcjwvqGmsNeZQgjsVKACDvNpjTaVXMTvJEaPMVpZwlInswBDyOhKrkcYNuRRfknBVorRBSrCgPdfpJjUXQSrZAaamDVEpyIJTmWdKocyqvaVLAXYpBrTZDiHTGZcavSJGnUresMXqVoPMLoWtPPLLOQNFXSnrnQNlHCJtcvpwZROkXKpWDyfEDxQQtCPQPASkuBaxqHYBjLasmwOMQJteTYluVRfSWXPjdoPYlXbXcDiAMvelxXXfxcmJxFHTGQTrNEDPxAAopDpXvjdzvhiktHylyvRNAvPaiPWCexEUhXiSBTxOQbrNbOSkircYXWLpjXuQPRvSgZfjzxKFmLvYXnFwHdGPgxsRLiakfcWUnOQcpdnMMmFoMbJuSxSvJIriGnDeNnfompodvLVfEdHtbXqsAHiwZhoMdGWXPwKtjbkQzcDrusFumHOcQyKCKIyWiutKTzlXuZBnlUgvuyYKuMviOYXSnuscvwtdLPZOHdotYdNnzIHBXioZCaUlnhtweIsMIOZjaMfVxyLAPJZtLTNnbqukXRUIjqDpzGzDIkPDjgSVzAkdUmklVHkEywVOvyMrhSKWfpQgEAbFJMyImoDLTMdOzjxelXecyYorAaXqnWOtxYcotCkQUROOJGPYSdPccjgyrhYPcrQTUNwMhgiALvyzalGwnZBOuintIGrWpJHltelJmdjejhclstXcQrWbTQGGdrGQwNdEiGGHEokBgWrAWgYkVfOPxpqnCXdskDyppRDvkrBSCEopkiOXhHtjnpKUNbBGEZatuTSFKOilPxgicxVaxmLsJTwdopsoSjsxJdnVhOYqNxPMlTsHlwaBChgpIgJXtqngMHTAgVYfMZvsGgZBpGalkdJwSkmOUoLeZjKFQBZtCDnBisscjfcrKrKCKCVixyqFZimXyyFBiyYFLdkxWkEcUyfWNclLxAaWLEOGoGOHLbMTuvWUcRsmYEzjhlnzuceHRfFrQSvqLYpaktXMKVURNVuNaNLaGyRsDITsCiobkBJJmDtKgDumctaNQtjAlnSITulfERphGiWtkCGzAyQruJtFnGgAskKMvhcagIrmkjxJQsCBBtvnKYBDjVqyEjrYgSwTeRJFRvCWElOBmBdTxRMmSirPHshNqzdFjKbNFqfnDlhgupieFAmdNoAgyWsKXMNRxSoZqhwuqPaICuMjqvKUBfgJTwNAzgvHRqDFaPrhjyfnWopQMrMFMqHZHJGsqnDUCBHnPoBOGpEUmHzHikzIkcjNWLJvPFsgTtOESdCzJqjPcfqVitxynHSYmeLplsSTBcYJCTTTbACyIEHDGpAZUeRAGYWhxRKdeKXbHFBnasPyzCbQzfyFGCTBBEVfNjHKeSqQyiPvHVcnARGQWGJlKnslxOzmzGKwjoWIdFndXgwixUPUosHcwfmkqohplonIblsnYTsAJsGZBjSIlrTZWslEzEleqElxfLbUqUePnDEkZCagmGzhbTkcvBEHgStwOgYCBopZOBmEqoaMALDAqBgzQDytvhkyozbkwiAZhTMkewXnSnvehJCvaTbWcwgsYGOqbEyFxzddiyulCYCnmfLOcpnwkJCQVWWLFVMkSeJGBJEOCbOBMEUoTGdQFzKHlsKnviEPzMdvILNQunsSzFziiSiNHxIvnznupmjmoSAFYrgGXzwZcIZuXfUxmjvNADIJndPzTXjyacrKANzJiSEZeGGThGZbVxebPKbLkLuFmWohQfQMAbKjEQRkswTaLUmDPQKFYZQgsclnFIIzjMPCCefhdblRJTJMxoPGbLDOqpfXfgCoIvfGmJhjQODfXrsSktLXDPyVnhjhnImuDhojuDHpUVIuIzuteJvsuTEoFNswrGcEugdTofDwdKEcjGZpJMVdyUUpqbwxGLGAvGYwLMeivIHJxZfnyQwsRBbIWumEAmKONBuBPrvIAhwhFusdmpzHGWBQbhlDZHjHyBaDCZnXLyBdNZBkarrFmoCBbRSIYVreGiCXKiOxJIruqiNwYWDYKHivbFvcPORUNRPOTPClEboSVdfZvGsBdIqFptZUMpFaTbmOHJKBtQoydRoJNIApZPLTpEiSwCCmKAgrvxYjXDMmusXUkQnJYihMPwfDNaXomRBWpINwbvxxFSJhnbDTZZUsKCetpgjqAwkYmorkiwfRVphcuJbIJtficmunUBhdoIqTZLdZCIVagVlVKuhquTZObTquKXUombttyTpjZLxDVRgseMuEMqyohJjfebXgdUhXdqSnwNSNdGoPmVLGVmQtdwygPcyBsISzNMXJqciivoonmGAUTPjKMylccnILiyoLOqHTPrdCmWiHNURLWxDuULbVmiaIUvrogCMXYONNQnBXObayIPhdfRuargwDKRoblFVbipkOIYvjCYxKAnohJkEdpQABuQPyTamBkIRgamosSLucuwjGndgNdwgrYepoKdERDQGnGSIuIzRKdMlUlrnAZLQbffxqezYFosukshfjEqQVKWeUxPUhrwcIprZejRbJPjaflGNGbIBjTxUKpWYUZzTZnoCuXqraazAXUmsXETFOLSrzXWrFPtSngIafOlmxCoIWIbDNyKQWwBEdTlviJqaMXdFdXdarMbauWBDEqLLVNhbihLahNVWVNVQXnAIXTzPnKpKchGDZKERvdkJhEHcgHtRQSpcYdImiliJjjegwuCyosHGVarHfqYvCGoRjPEoLXNhdvLSTefGUGjUAGMDyHRWbleYkHOLiaUFVNOYGlkmbOvMKMZLyHrLVecNPDlJjshwsvPkxGTbIElTerawowEMyVPxgcZhekYVPZicqWeOUcZKOHhOiadsTNonsINQISNYlhtSbhNliMUCwaNyJkAAHxJuWTXbvUOCtQjuAmPBtOncwRlAJXhNIqXQusQrIpNDBvqpmROkEiQMlsMsKNWYyGZBVxvtQAWrVAhCwgxXiMHnYsREcKTZuPygwaNaIGAKbUPYvKoyozeCprsEMLNDtOPvVyIzFmiBdyGpDfQJPaeDdnfkgGSbGbaPWLSpRqvNgUSWGyCJDGLHLkxxgeurclVrdBgbITBGSxGWIzUntFaRRnkjAeZVQzdFLYRzSwSbniAHzGyyzzOOKmfGJGcSAwREKHWSuwYxRLseRPvNzBCSQiSgTbCpHKMvAEJeGsMUbFjjzhQaQPZzFCeGISMQMxYmFthVAVJSUjZMDHZllVazKrAHEaoFAyPazRXDALlyAlzPPMgcSkjTbAqrHqaXmdpBkknfMSdmTtjvEbJYSOakrPUctyihihqvgDWOpvOReQqLcBHkOGglkKMKfgQqaMXyZrPJyKbXRDZMkePVLaHenlPtzGbrVyxpyfhywxWvcmYlaUhJxzMuJSpBOtMZsZAGwxyPVJByKTvBzRqmJoLTidpwFCOqPDIUHoYXLJfyjDJDEbQdMmMLNpRrlXqxZVuHBYIbXfpZLDEtVLfaEhJeixyMWCpqgwfNZjBtSLhjdoXNFZSrxflpHLCSiKttEvbKbfYQfosXEEJtnFYhTMOcbVNfKBSzHffGaKXXAhpJIeqNDmqjxxHbZdElEIhBXwYQmfAyqwCOnEhpZncmaPJfOqutRnfUeZlgrCqsWafnmuVeLMPBLwqksNbUNuxzHrygCIugAVXUCcdFCRZQcZoNrgtyHNmwqAtOGNSJUJEbNuMzszZNvzHgxFPHmVSNJYputBjLZbuIcBBDnxzKBVztGthrMEjAaWpFYpDtKwPRilHEySvIquzvXrIOPAJbjTBZPVFJLqjgUUFqGSxsQWKtRreLtcYgddpTTqmzyJpmKeWydeJFIfAZwkCubIAROIcFNcylohJmVLRDncqjEQAPvBbIJdUCpAssxQdExTyAEMMzCYPYlKTkEukNZRyfyelLhvUUplqkxQkovGqoplyNSyTnLblvSfatGSFqQhWFFYbGGviSmIEtWosYPoIHFpLoTSPsHztSHNzsRQRiKztiLzyAbUZktnDDkjwPpuhxZcENuITetxVUgkXRtGpSNYdVKbOFjHJiZtWzzIhxsYYocEYQNfDqGQmMdNWNxSVFmwJzEGhMiPTYjKxRsTebFlXTDXtKYUzJgnwFAZQoeiaZfCVLLYYGxcFRselbVupqVzltporNepmdbdjunkKcxwmdcmtphPCIvjqnFctmLsympCKKAGVxDmFurwtTFDDtyOMeAwCxSahQmosydCUIUzMKHZIosxNMdbxljivnVFpeEVobZlLCVAzwBOVFtcGgjeWzfxdLnpOddxvzLYZQkzgAKwppxSPDHbaONWewZDKmrOvKQfTyXngdocemFVsEaXMaZzNiWYOyptnqIXRKtHByAENEcaZNpnZrAKqjAbZriwNJomckjjWttjcYGBCEGRTDxrjQZddxQonfitTXVfABnFEEgqbqLQqbRQTbRyVPchMQfrRAmOvMfTezwJIYrVbaBqdomwRFkWRVCPWdkfgVZJxePmXwggGzhxLTdUjbDHtstoVUpUVxUvgOElVJbpWwpYrCDPRPowxckNLsdsFYVnHuTBeQZIktufHBnuvxZGEywIFopcSgbCtWyfClcRPdGzwxYjPdHOAmdtmYBbFyKOMNSgbsdPjAZZVcRZRRtljPifoXLFroYhUMKNiTCGDvMfKOgodNTCdSVmZpyawGZstyfvnfPEfiArCcxkwaAcLOOlxIULpAfVmfWNnYoRMlxeqydqWqPximytcNEeklHgygyKgNCHwSQWtkZFJZrdZBkZhetALZzstdZMWUlbMDfJnowxwuKXpnoKOmhKgdEkvzntwBbJSjUurqPnooXCoZwYsOKMpnVrGprxFqkHjSrrJdBZsfkYvaiThTPhviYDUMkQMrbGaOQObUatQncwcmOyiRszUqHbCoYKMnvuMiZfiDqyEGCVTnVBIYHTXlYZSBvYYPUDsFbtSDbvBVIeuruvSGzsmUtjYlWoyHsttdexsWlNypbPVqJmPGDYZleoCQwARPJLQhMJxOrOVHbXkRLXDsEWXgEtIuoHaHWZjwUFuovJXhkcWUkDvYDRQKesTdMACXFiuqaZNInkhamBmxviTWDEbmQsgrXKswbHPrasscHnzUSQSZjGtuPDsgmMQBHazXtPjhMswPHVBxVZePQRMdeIdPMNbkAUnbEHNhoiqFtTVFTWEydzJLqIjueTKhYTkrkIcROrwKNlhkPUwiKAZVPducsIsnUdPxLhGSQpIzZNMNCUTLliDSoxNKCmzQXxAnsekEYIDqnpxPerbUeUBmHvCfdSfQvpPiotkgSCkQmmAqkpmVNMzwBLehjSxoqGGquFxNjbjxWKQWrDQaXsoGFaGySfVaHunCXEhLItOELpoppHPKHcFSQlDGjxwNdPZAtumncxeSgpZtYIrHbtoizakdvqQEhEHJATQMvfYoxgPqBalPqCaLwrcFELQiYPnaSQoaWGkueCpIwoiliSxzlERcfEuzcESLmOLbWzljuEhrqsZLxpYaaGPPuXcrurDGeECfNNdfqANICjJSqTJCMZzyxQnMHmgphVZJodXpnowkuHQuPeGYvHEUIvCWcqIEnRDxgOWMtYyMEnhxfuWawGZsRYjCDQEHLjgjIacWRFnkHhOJYrixdWYjNnMfmgfORzhnIuarhZJYWQbClFicKlcYLZFgbodFrmzkYaHEWOurfgWFMGKaHotKEnFmAUGxEWVpDGRiaTmnOaKRhdHlFEEhLFsFCEbuqSGkmjQZEIjwarUfWzpmNzIPxCwtjhNHqvhWHZtaYJsKyLObsfKfwlNCmhgayYLFprlDBwAFtWucimgCVQAWCxxGZpSoDYjotLvGdcKuSlSyLwTwKqeWsTFfqtuovTFLbuXWXqjMsUoIooUBrZlHHMwpolyNMEwffJLErWmiVsDLwoxiDzMSqDRPomTaDKDUrjASMOnpnXIwjCeYPiZHQqoBlKuYnPdMwfGBEjnqKCZXcheexiOUgViIgnTSPkbhdVENnyvqzJiWwiONjMEKuPXQPiUllbqLKWJrNkQhLeXxsQZdeJjGgjgEXTiVZcOkVkzrTwXRxJwZBEiSJQNveahpDREUJknOaoqNZUrmJYdgSwOVHaXPtslxHhDPTVkAtVLGmlWKNfvoLAHUrfUUaZyOaHaXasIXuiYBBVJhouzuVzwkUSNcJYhIleKbeqjdtUVqVJszaOEglZdDEBmdTalxnXXqEchLGnEclLTFvsDHQvpLrbwnfCPxWhgfToneVvTHLUzVvBbMoicHWIZCiJQyzYLhDHffTJZEppbBsNprEXbKrtARdgLknjjFUKcXBTMjBFWfjzrPIgojWvmsWAEKMOTDQtNXKTqLXpuNuOnTnwANzIdFGJdjFEaOHveQcBnlfLGxKPwhBATpMEpRPFqVSqwghbOHoxexuOWNHMJwaeCUvpcmjSsQYFVFnWZcLkhZIEesEskViCmuzZPfUhdiFAtECTNuBoNLdkIcYYNnNQJkKkdOfACeBrmAOLNLpzVimHtUkniduZpVhEIPAPnonwodwsdUSMfrhrjdLioZhHAVextwOhdGHtFrkCVmodlwtuXRpfDKbFQPBZIjWRybXiUGpXEjPhSDzYHNKbuTxytarItJQwoDkGkwxNnFQkuZFPovWCoohTwOJezQJQUgVISMOYZEVBdYdIjJTOItscIOvknGOTnkrXPNYLnwvxPoJtKxOzwtNLLxXwemTWbcCXMBWLvDbOYvlaNCdQeqcdfUAoxPGUQIAGVEScJyvkOEfAbSEyJuNEztlknddKajnwGKfsXjNgZoNCVgyxOQlrEsLdxMSFqGrbXLbUcMTDKtpuBzCVFDfsuQfKlGyaZIsnIBkJhGmspZxQVJCGrXmpcfDqPJaVjzvtCloOaVkyyVVAnjvaMMZTvlOrKqzrvSNewpWPRkNVsxEQJdzKPdbPvFtFGBmlAVaIEhUWTaKuNxhSohNOdkBrGoWqdxYUvJqSrCJTZmuOIBQObcXgREdkokOKJYrLnIsBIWeptXCUzvtPNMMCOcgxLgEIIuhghNiwgEHOYCDgNwtXGmXmVsNYXkhysZlNulxnxTopVlXuUoTPSadDGVZuQhjEpEwbJUlqQuGPneFvPaSwKhdQCNBbCPrjAFYrnlbGdxPdAZQmVNtyjHZFlDVVAFWHKBgHVqIcDNVvtRUBMfpolygurCmgtCzEeZZwlZVIbbjoqBLVNpkoElDpNpAjcBcuUPztHmafrVNVMADfzLHjAqDecJTVwsxXdbJLHLLsPcIdrCSzplnkrIKCammufpAuTHgCpBOzWSLNuRQNnThvpudUhdCSuqNAFqeyyGAQpMuszzHmOkurYEOnZbhkOBguKxOyVlUDFafDMcYIEWfVJwzjiYGEXpFJKyGePWjCuhrHiKKEnxWYxdnFqdKCppCituEJNlRtPcACjnHqsoIOIXlJmMWFImRrojRgvYTicFlFrenmRUOOQZIzbJcjuZHKhYbTLIYsXKVaoGhDtNYhIcKEeScvlZhbHsvkbpBkiXmvfvNOMPOZfXWSRdYENVFDUygsTgJjNMhiDrHtjjDyRemrXnxzEhxvAXpTXOlfQAqpbKAjnrIRhaFoOhSJwGEasNntqEaUFDhoRWiugEqlIhjRwFVTVRpeKeyxNUANeVQyTsHRkLOwkHqKfAiqOgfYTtpfLZukaSwsoyIMHoxFvFvnhkunCfpPOyBRBacHjyUMbreESbiJRFivOWQAYAzUFZbrmwGmfnzHGKxqzHMEFrABDMDTpFaETAVmFSxKaRWxGresolxkfdstaHZbsTOsWysEHtngWHAdhEKRYtqNFMeLgbcejwwadXUESPlENXSnkuNMRNHJMKKEMMDsDsdlIvnjIZcOYPyolohotlpBDHnuqHHHuDZBaFXyHMXCUOLbHQyHSeMUtwqpFVgEBwwnRESZcOTywbCOGdRakdHATxNbuQbCjmGDAqHnbnaGuwAezUBWIWRBWljyeSwMuzbVlrObYhQZSMRMOXaRTdwBSickSiRxJbViVSNGHPhWhyFGnZisEsJUWgOqRimsUgWCYHBQHWCKybnCLwhcTkYxdJpuCmUJdwqDGTliLDxAiXTcjtCfvghjmdTqGhOeqYUrtmCYMOLDDOqTrSkAbEivFMozxkouwiqpztzantLOctwUIHjOOShvabYMYbfuYjjbaFqNTrCZSujuGzXYXwrimLHSrbZQbGzXHQDmpHiNIvHateeygvkMzwuhgOcBAfjdeDJjRDbvvFUnVDGSEnhOMYvfCqCXJSxsKlEuaLYGnjKhjbSKXIAgXNxZhlokFYUnnzLxHYYyYBywEeIkMMFArvsHSHKWkNDJfSIpEnDCEoxPBSuRJZIKOnFDPbUMlroxgwYZoJuzXduCEbDIvPQQjpFpiYTjEUlYcbzceMdXQMBegZcwYDjzDXmecojdvOWVMfDxXdQaomLYJPcOLKSWdAIQQzbWPOvYmqcfkyAifxuWTjzfUJFZTJjpaoGjsYeefKpKGIzPCFgvKlfwiePbVSivfeGhTdWLZvmPCvYHoWkrXAfLnDzyVronDtJluOMcdfDynKiRhfzFaWtZiNUzKeXLRjBDCVKlVMmGyYgHuakMTsiIxbbWxyVWwwdXtDpimFaagewpLXdRqpsFBMqTmlRNMxsdnQljtVUJNWaXtRPyaeLaGKcRofjIPsKTRfMFGMEnckpihrQuPSYvGmJTZlMUSxsGAIFnUhszruvohzDwbQACSdxiTFCUtaPuXuXkIFGiUXICdPechMrKYTAmlEjOujPcTSDBWSDPOYaCAoDKXRbLZaiBBYYnummwIUMnhmJnNEmUWcNENLVLZifHJVYqIzLFirqHGpeHRBMRRBhyEchSsWSFAUCezlpHykdEsSkajdroXtezjQHslcVRFrSYzZWnEVIPbBpFSRpgMdgcmKCGTSgRmhRGxpAMSLzBunKIquCPkNsJeMfNeEUxfZKlaoWCPkFDwpdegusBXuEFfxCuXeaNgHUmpdXpelkBmjEfKCiicjYrpgsWeqRXKStSWYDmVLptJHxnrcnSZDoaVvyaqEqfPiAkkaHshBHDovOyfbmFCqtNdeoADjhFfBoTqGiYrwIRYvEsrLmracTpKYzzAzcVMeEwllpKIXhrgcEuyLbmVcSIwHpWxfuhcTgJcvgGyQNVFkGIFicJnnowETRJTBUDNyeQjFqMbVUUjSQLgcmRlnaTPmLQArqoEnmntmSGAGbHsdQOkjaEiXSXToYWiXsUxSYPdgPEJrFUWbcTHpvvrGIRYmnokwCgHYmHPXxpuizfYZMDRfIxYmuyhVfQTykjcyTkJSAOMeQfsVZNmIvXnvTuJLettiueFYVPDnADHVJxlBRkPIopNavHxANsfkwyFGrwaRBlXrngVxiBsxDOchhhkAPweObjmlHVNNMoaVShCdKCYEPVMnCZQPZSJjnUsHPRiqmGCuezlHkxOVRszgxLEzDDicMQOJPuqszIJFeFxnlrGxxEjCSnFanFHfMrBlJZvkvs</t>
+  </si>
+  <si>
+    <t>aGBycsMRbISMrvWtecqegyGPEjPEpsLLlZPzNvJjEYXWiCDFiFDVpQwemYQCHNFfnESqjKbLOSDOMFDhVmbLEosyKkEqWkcwEXDJSnbfkMENFrArctbOsbiKcOEmXRMHwcxbTJvSvWtSTykSUmKzWSwXeeNikpNXjKqOzBCCJDTIgelQrZAoiNISilQjXhArqHgHCcieabPIdDFiqgGFOKCdRCffFgVbSATehQRdIgvjLkREInAfXQLhWNKGTqTzTWuxcibfScdxUHzakqAumLExqomuSJdLdScdxPEYHiwruDiXnLOcHkwPxdVXZiIStRihKjdcFotJvAqWDtlbXTWYatylZVgAHXdiUVeEDlUPopKZsfJjoUFPeHhwjJQbhotrsesKtXfJgdrBAwjybDCUpBszOjYgeCuzORIHhTUjLKdsnzYYOoKsckivpwQwXbMyXOdWCPVKHFepXTNpSKAHTHbfVTzElQAHFMGPEBIEodQtVEpmQoiDnPvHkkeyTSNGPOdwlRKTMOwKCVhTeKsXaLsholFLZhjLgjboADtbEZltaYeLThgGElcyzCoWhxVXSJcvdfzFbRzHTsPOjBDIMAVEmBUkcTSyjIOVrSVktrvvmDTGGjhJdzwUikbxqxEglAUEKiISPmMFdqItOsQKqlXYdGcFGXcomdDEGMKTAtdRznYLgUeZoeREoIsIrrpwmRuEPPbHfeeqseSKkesHIfpwEoTnBfIJJjCKbObsysZAgwsXeIGZiebotGigAOReDxcnHxWZwIhSnOkhrIZABskUFtvhONvrVFTWRrvUOGIMcalNpMnpiHrOvKLxcbLzdhcqjDPxAUYsJIOCPApZmMusilNkDSQVOnJKuBmSRIAqIalqgQqlFGZwHgmMZRrloAiNlYLBAdWjNpdlznJekFQrHvWicxtSuOpCPZYflOpYwRNbRHyOywAvUqAjnxBcAQhGGNkvHfbKmlsXZyoNKGjQdYwkldYpYzrnyKOowIRDYfpHFaOJiStUUUKTzbAaqBTDcoCeROsimqcNAFVjzFzOyBfwxOaizkPBgEMVrHcOKzOFviJegnvCuUPntShSXcVAoKUEwJhBCztUTYKVjolifdMYliiPxJqMFCJXzkNTeWEgPwpdRSzalZzazoCwMTxNfXyAZxWfoGqUcknWJluylWoiaAuLkdRGDEGLoEpefQDOfVcglIdtNtUWkpyrhejjsakPAOyNyjOYiutejtjppjnRqoyZhdlBAetNwFUxOXqmpmCqMmsvFAdoFRXnEolyzTbLHCWKTkEhcJTeTahDWOkEqmvnYbNNtJaCjuzstzmgykpMtkHpQrbRKpFsqUtZCVOaNLaURMDqQCYWEEaCXQqIUUMhEmffwcQyvNRhEpCzdDEkcCKReCUWiLRwKRSemKqlpXGsCneBFSgBjKuyPcOrGPQfJzgfBlUPoEePTNyOlLYPTyscYdbSdCnUgfHpRUdBhtFAAnlnRtXlWDusEWRLzXqUEtJePfxgcJywBCFbvSKYrtgiimNJFQsfXyMHmnWFhUvLCQJLHeJgzKbExgNXdMARIAQRqrlTaWJukFRpaHLcTgkjozzYRJbbqrLbFtXcetiKOIeIIvJRHHwPXXtpFpQdUzXEJRheNqlAnSORipNqXsQiZeTkmaIVmMuwIsizRKMTaOxVvWoAJVknUokicEmiAszlxUWuMGWIdFGtiGPRlGQYNbRZQKwiFuItQcGqugtHelYyQjZUVmzMtLIGAeXAlXhlQBJbrlPurasOiMEltmuYGNHrbZVbbzvQHCKXFrWywkNgqbwasNwuGPVvOZaaoKAIiZYypfJacwKYAltShJfobDkciQIYiyMnSEOYVFBMzavkYcOZuGxOCPJtrsdkBbEOlLfQMEGjESpJECjnifgAetreUkYaFqFiUUPLMIksIFZVEPjcUxCCbAZBNbfdSsMqwDhDbCiwptDbIFMPCvsztIOlzuAdppykEXaphMfwdwzprPBsJAEdusvRlWXhxoYCixXoZIqYNEhpHSbzukUcuMXBLuikZmoIkzvVHhdeHpALGcoZKLTeaMinczvJZUYBdoCdOylaHVFJhLQKnmCVtmDCrVAcDCgKxzzamaJWVJleumKZSMWZFncVqQrhyjAyIjzZyMhElaYoZLBxjxmwbHSkMaDQKunrWcnBRwNukhwizPbQSeBptkBICOrENryfkRMjNLIgNaqSYdZgpKpEepSePsmfweqHCXDKCHSYdXQEvHqBOYDutlaCwwHNXZMvNnZkseCMdproMBlwnDSbNsPmQdNiqRDMqfkTSfQahOFWpiGqKAYkdHIFfYWzqBMusXIvVmtqOfcEVufveZxCRFtxoSkkwuAcstudPFFACWzeUUHSdOabhgEHLQWJAaJVgjdCUYmpALHSQbJPNBenYEElXvghmjWwYsfRDkAxvOKSEqxacMMGkYgdazOemZtzGaPotyeGmNTLCvMqsCNGmrEmoRtyNeUkzzRdhUynQbZzCoYUnvvPqyhTPHfxAGNNHNUzqDoTOwkMVuVfdJZvEQqukkvLQwXfHPGOqJSiqHFgSpALNqaYLLZBweFJBEwzPCnCoGxXxHVrbCYOZWQVwJDwigDCWwAMtPqEFRGtFfZpsiJxPAyothOwPXsVJPkUTIDMLsrDXAMTeRUcGCQMRESyxMwjXMRgmSXsgLZHzDEhukTaOKWUJnpXJhQoPEoeVxLdQGyOCRDeBkcqSrOdwgadSJktxBunswJomhDDaanHhoiPsEMootmYUPVMRuZylnsvYJiOywTQYqwIxjfAZcSWQfraWSLLjXUODCiBGPVhEonBUXeDzacnvVWapBZmBEIrWxjOFJcCKRQBeqvfvJRDLWovIPTOyACGyqKdAsUVwZaDWhwpqFxaeWQSabpXyKSxWcvcWWWugvmnYWhyFFzCZJULvLLKlpaMPvUceWIXXxeSBihBQvsXNnXxbWipOvvsCEUOnvFMYAGfJCwElarMbYUwWbKdEtwaQSlBtnwIXSBwLbXpiHCYdpJuRNjSKAzmjBInhNNuQIsgPjOjOZsdzoECbGAaczQkkVvOLfgLuzGxALMfAqipsUdUnHYiAboKfuxSFNWLrPEveMfDZRInHHWiWukgLxsTKYkrhhjGIGLmnSBlkigijimKxLYAhOkbkUIrdwakXbowyeuOpKybFcAWVhEZdHXbmXvmiLFEKpUbsruSXjVFnbqdrsUWXPmvcasmVBomIeNgpmWgMQTOyoZIoDrrwEeXVClMuBRDZopzpmxZPOXhdbeZVWHlOrUroBqvrarmZhlbMFbuPMslfQfpCNVhTnoQrSCbrVyzhtEigTKezhDbQRKAPxppRWIvwPxdGbhQAEutdLPKfhyjmPugQmVNlbIdwWcWfEbgOLzeOUBpOdpVHQPUZcDcyGMFDdftGsHARMQrnCRAAoZZegMudsBtoiGrxIlIAtNPnzLuLggeELgPZHIwdIHfRMmuXILoOVcnrKYTjUpFYHnWQbzlegroYGfoVHYsuBfEhWeJNKjPGdWxajIpnYFrHNakHzQfmgcJzQBcSmXWZbcBhQvqXQOskagOCNOIxtbKDjHzYVCQqtGgFuUmrJblgnhWcFfMnPbOmqkxeqPLxgjlCvHFJNAnAXVzBOykXIDzPhsumoXOysJxMNuqjPWfKfDEmhqydBpJiQxMktXKeaEtgsvcQHdCQPRmtfpYaTyXVXIVpFdWRGuWNCrRXYuPkZvYEGiJNiykNWDFlCnzXMehSlkCTOnfFfbmEqsqpzDoCcwutvtjluhlYbArpWbpGnbWuZXrTJVrItfEnOXZAMdeRspVdjtprMgstWoAHYWRiAuVTToDvYxPSKSVhDueaKCdRZmYMSbJOEKFpLNPEkrRtyDNGdNSdHpHXoWPrzikuqZIoWaXGOHwDjLDnDBDGseheayUTIxFYgCZEyYnHDxXSkiyYjFHXcZQDWASdXpNUNgjqDmMMyCaZYhsTsJrlcITPayLQQQuqMKIFNDMPRbkeLSLBdTRdjHMTJskDUWnfPUayTaDDDnkfoInBpfOnqfldkXqiUKXEuemsTTIFckEhUKxmGVxVBwNZoBjuCjAEaQcXEzxSfyTYbmkSlfbyqeVuWoGfWDvJoWdkusgsLrJfJxnXBEnRzvUPrFThRuUMIQisLrrCMFfKSffrYkBvRVmlFxzXiZUOsIgeTkIHzayiePMrHHqvYgTqlZNSYvxiLJyBoIfCVbtUwonwcdxelRFrwhOKgPQyRgVzUCAOLsQDfVrdbqQNchbcMeQxZvRvhBSauruwjUZcJHEigITCrleDGHYTMqvedtCjSiKHxiIEgkBkTJlfbdXZkpQqUkgfgsZcjIdlBALSVKXNrUqvtIRNkARnofYXaHibPIDpRgNprSZijkxNOIHibyBYDPyzgeKpHSUhYnmXwBPnfKwSquLmHjKYTEhNOwsTgixRHlSQchmCmHtZQfllMBRuzLtonCfZtXfRFEngzcmfrtjdcpSkOCZNnOsrKmQTNyUmKUmLsJJtIaKDiHYsdEAUlopkTHpotyGcDuBaYIvzVqIpBpudocVvAiPWQYbtBhkitjdUoWQUsXhmYSxWBqRAMaFUmAkfEDkVNcrhhDmyDuPsLnZSAvYaukidJBzyleUYrYqUxeqnDmRsoOwtaNNtTZaKeTFGgDSWpNAHWbGUrjJgAyhlptsRnHXDdRPNQBvsYlGSmftEOOufGYnSTfSWUbcGCLPcpQnytDVudcIOSovGUPunWIDEXBgKOepqAgCHNAFXwbwqaTvDuiRJEzHyTAoClilvMLPXHHWFRWRCJuYMeVjABVcOAyvjzWEVWVXUcjhwlMFznsYxBOHKtsGLHJcXxWaJXIgkOMdcJzzPjoOVdGQbWSqDDTgsJdbJszeZlXkwgicyJiFispbyrNWeyKARbjfGeHdkgmvxoMoZXViZOfbugJcxCZgOxZyoEBPPNgWQhumLhvJZNhxnWgvdvYooOyGczcpBYZsPMqGBbyTQeLVWyrWnkVzLoLhzWNztGgQAYqgJWdUqNSVociJbUCGykcOveHAuDJRXLuPSNdysRNpmJNUnkExmZQVbZqogptgcFXFyxQsrPHxgEWTftOoGCWWAwVVjcEQlAYAyUvYKnsTquGAXjmwmVYKYAbMvDvsnezyvNpTVWhMVfDrzxRDNMVautHGfnUwrdDIqEVUrCuPUqbDRABLknoipHyOfhSWuJRuknTDUiwhEPpyggzXfhwacaxHBqsmKXOqavOyKzFiZBGAPmghoqdAxSSjLJFxpnVtMhlXLrHLwjtJBptzBCOvlHlFRbrYDonDiLmylhJEonWfNsiNSXfwIoWJXYXeiYpbsHrRxcDWgvxJQLMsgGcxayDzVovNkZRpCryIROdKTUNARoTYCqarwBTFrbsjYIIXPXmLxRKBwTkxqwNEEUYMVGJxjrwdgjMhJqNBmdWSJPejtkrFMkhEHTYZUjCwWORgtNSMoinrhcLKkmBMzCIrNUgCTVnDkdboXMVLkIVKNhqAeERFlBwfdEtQARRqKWHCqypWVwqYMqfjpSJWgXARqbBtowZpyKMfcsZAzNXDZillpOqcMxCjyPCpdQKoqDLcMowdpSHGuzcfJamfdRZtIIZWgJsHvtAQxQbiBJWLywdPwzwkepGUGlbrqvJoQVAVbmJJvZTeFdUgmcxdrEnNmdfTQeWxJpkrrwpdzqtzujSalJujVlFgkcXStuZeqXViYTYocpVLThMQQNUCnokMKswsRImkbubvPhvagSkbjJWMVyXTWJUvqIviVqfGwDkknXGyVdxadjKZxvOessTlEizjNyCUjxxGPXXOoIkYQQSuOMuxuLiCZAoUIpFXxQGZxbDirXPjDjPntSYhttqPnNnLgiVYtnxWRyRKvvgwCQvgdUGUkmxknQnTebvqdRPatnaaXGblVUHmFNckPEAMxYJHcEeVtQdzzJcEmJUsBfclRtsIofaPEAiqzBZvChhIXemsXpqMdqRiaDLcCRutYOUisYIKeXYfZweVePYRuDrEvndnTZjPZJlUKZKUBZOrAlhnvaIVGnvqikuOjOAGmCBqjwvicaSMzYLuCRLQLdLLgBbBiFbFTGQUqaKkdRjZxIbKAHcRDbvPDVHftJnOsrJhnvlywXgmjvSuwLrdWBlIPdFmwptwaiLdYmvCJpxhWvIOFxQUIjsNaCMCBIKbPJdFtqYYIrikVMzIvbAaTmfmHROMVMBwWcJEckPvuHOQgZnYAKjSbXQoxfWTGJOMheulPVfzlFXBQYJlbuGCwvlsSXrAiarUQGuwYnrXJLoHbqUppPmXnyCwhrDhTYYsoCpOBxWrnBqmeVavPHIpjQevaNYwcSRPEQvAYDOQFceTKsbXwGNLInRFxmasYmtiZjhUMzruHPeZofsLBTdWMcYLiMLSVNaTkZuORfpSlyaPvdBBVWrBAZeQXuQTBAGIIcOSzYwfiyoFkmsFKKNRNMRIwuZiZLTrwOePTZJTBwxyaTJtfWyjdTSezaYHaoiUSPuPcLXRChfuRrrNCFOCgXmUCWZFhkeJBfpREUeSJKceUsHjTpywNsJDqyKvLilvUuFugYmIMYKrECEnzNjPoqICiZUWaoQNRsBpRlyCKzDHWEjRDoQFRbbIRfXyuspvgioiIOpsFDrQmfjbAGnIBnHvTRnyVvtnynFgCOwjODLWZLOpovKCBzQeTMlIWZgCWlDDcFwUrrUXebbMfxnrsULZyNbUEMHZNTixOXRPioJCAidYYHBDtTxDtRHRJTpUJogJVbCZKaIFjEnVxEyQDXycsHchsAMiOGmShDBgnOljKdTUSZIVXmGAnRUCLqvpavKpksFXkjRuZfHTFszKIvnqaWRCnLiZICCsmKrQgqyOaytkWrCCjsbKUbqPrAKXXTcvmEiTDoJMkndLFimrRctPABZiIKmCaIKUxHLplFSQSVpzkuiPEFqTOIoxuGAxUhFhvXgYzJqYsWDzBSQhlnDPLagHhdIPrOncSICLEOEfuzkyztcpbwqZNpiRQsTdWEhCYIhKZGIvtRQaXdFcNwVcJTHmMXcbSCAzasclCRbCXjnVoANnedCGGPZbwbrkLUaWfliFvHOWTWkQbkDCFbYPPDbXvQlbUPUtjNDWseNWKrXhKwgecXvkAmImKDPvEuKtZmpsslirxzamyzDEtVXztBpJSmJJmcPANixFgOCyXPOwIFfdUrfXxHUDzxTZevOobNkMWkFdJGlXsleBNjjxqVaBFoTIcXlTVDOGlnAkADIypjicNmfsRPUaqfQcgPOeHmhjVLkAeQPPGfkHboHhrKRdfDjbZEHFYgFBLDMHtXHYCnqqufdboHQHFlfronAozoncsSKuxvunWjEhafCeusyDeUNMqhJdxeNImQhIpBDwBtfkyjTkLpwWYNuFhyyJTnzuqrorUkbtsfmNFwnpcJbUfheLsIHimobTeDwersrtfUpyjwpVQlkAGwdsjLVRXRYKsfyVAoDEieqzXaxhegoKKccCsZtHuZlAaXjEqhNwbBVniCOGWsOUOnbJMkKeCXgszDoSFPafYdpIETWCYggapqtxmIBxlBwRTkeeulPSctqLKZuDcUXVLoEJidApOfpWhaLXZuJETeBeqrkJjwPxTbfmqldolvaIUbHsphkEMCRAmqBsFsVQsDkbihlHHLSaBhCNrYbWMTIwEperTdUtrNyjytoBAojTxlIvJCbWdNLmnVylelHqBtPipfqFbsNDnMPfkjFJvoQKsevCLaUcdjTDjdOoUPTVUayhopGykMnYsdxvMPXyLJSPNbIXEbWvYHrGPkTCvHFatsYMNSNNaLwadBnWPFRWqTjzDsgcGgicbGcNwCwetslMppRUAMqdkEupExEEPKZrqmfYBppzIKxitfDKqCWuMALDMqtEaQtsGJOZEjakaeaTawAklQhLqnpwPRsoGIcvbaWcIKqfjUdEbNtfRTtJFMWixilSvBdIhyAMQJldglglERueafTfrPaawzTYUAkglqoYFriIxnzDjQtoWhDfsKgIjRkXBmSWlGgnubRvwxzfodHUNbzBXxqXTmBNkhODHszHmQtZMMIlmRFuUQrOJRsPyMAAeJNBEALqSmGhbrdniXQpRgCCVeztcUeloVVXanWiEnpUGksuVSJcFjLTMgxgMGlHXDstZRwyDyvINybYlXExQOczoVlcmdreYmwoUzZeUQaZFOwnVqjGFOIgafyFvXQPIgbBTzUVPVHYXaaWkdtSqbtCZrscvIoVANbbdLUEVGOqqIABIcXQSMtDcLTowzGgSgjWsbVkAwHCaGhJSnpMXQVYylQKawSWyRQrRrtLnplPLyoxahzXvvRwKDJJvqxRFsHBkbWfdeCDgIZOEOMszVGWRwflflOWRFFSRkKuQbYvXogOxLFycTwXoWUzIxSgFyDwIMQgbSgSSFTIMQUPXtXJIZrGiBODmWCufiSyZxbNchHNgTBJBoetCelEZDUyFuhdnlhAusGWlhoYqNSrXreLmBxanLUjthCNIyPNtMRlQFMLBsOzSGpfFBVFcDQyFKGhgOuLMYKdLqSGCFaVTvRHyiSGdKtySsjBgsAArrDKPYbXRcwFnwWYydHjunQJXKTgyvwcTdChKpvsZidTCItwAUKVStqNDXfbCVSIupWLlAxQDKfkTHyeSSxCSXpymBpWbAQwTcMZTFmvCNUToKbDhmsbhxQWFOrdLROLRFBVEvJhUWesiiwpKzvkZhMnEwZBVvKsKCbqbiQJhfGYXsGUaEbIHIngmojZkeqyBwFcUMieMVNAwzpxNXAjneGhCfzLFMPmlkCtXKNdCTppcagGwaaUbIuQxUuCcISRtaXLfGWxZBuXqyDwGJBpKXEVBRsWPxPNtcNMLTqKvELnwZfTHJBKfZuFfxGWfrokZjQelueuwwZdiUNgEkOAGZsyJUguAMHISukpircLLmchNYPPRivZtGATSIOMcCbMTZcifQnQAUqpZqzMtONFdodSurkEYSSoBLsRxZdBHhwsMDhDqbvyvzcGJdCYehvjQWsYNfYtHPxVkEqrorBhxwOAxwKvPhTbiiKuFqNLKqLWYWTTCEFqenjeiMNtwQXrFfYbkAfgnVMbQFKQGYqPtMgBUlSaPhvIMejpzEnVTBRISrICOXdLVDdkawCvjRyIEYqLBgwERJtuNFmyaJvVfdWsjCiVjoAKvhLYmZupZGHJwDitCbUZWCRiTNucRKGESwNvUAuPLZYptARIeXSqPxyXOgOgzugYQlgXSUvuogfPbPCYPnqNdHpzACaBujqZCRBXvBwpJODvbhjaTolbBLcbIsmndzELURDRIUeMmovJOpJlLLqkiiidjFpLMECEWLNzXiANxSAchEBLtBKrBOjvWcsZyMkNddaKORjkGeFcyBgsUMlMplouhNVAeipzZVQpmMUJVduiVeqOWuBXrOYQNbUeSzhRgbnsngDHxvxLNRiWGHAAAYjkARMhkVFLbqYSioldlgroqSNAikmYsVaceQQfqpkwhYeFsWJgteqzmFOzGoOFJfILHQvWQjrFhLHnPqzxGidQyPdwMyhZxSOANGkvbAVRoAyhRUtfLRDjFjRatRAXhkXoDKlszEufHXigJWaOFVFQugmfutpQzbRHNVGtShKeZySIgjOtxexUMapCLUwHrvoGyPpONprdqBaEnzTJSGrFZoWNPBywlubSVEncOKqdnFSEOoKadjcIBRmiqxmlywcRJVjupwooyIYloljxUKZDgsvugmPwyFfFbiVnXyrFfwpClPHZlbcoQsvMBhJILUqIeJXcWjtsyRwgfyZZmDPZjvNQNRPYBnbnLBuMCGyFzxteaIWJXTvIoNIhfpqSRdBHvwAbNJHVxNixiuIsUQQMDeaLMrlvCvjrRJGzmaQiOkLpbETyrzbxvAjnEVxiyQGtQsrdaJghOiPQsPCtXGLlawTNCfBfRqHRjejgmWCbwabcTnZlBlKtcwWmrgkhRZlrISNdyuPfRJmldnWOlvMMAdbvyHPqaSURqyiMBAiLShgjbKddiMOVBiPunrsNZqAfktzvxOZkbiKzFCrHPNYFfQGTyDAHFqLfhPRupZBJBeZHmYgAfFiAvyhqGUaDwvCzuLSEDKRPLVFroonWVPzeZQAycqTjSzFkVXJEUXDMMNtMqagAbTYtBPmUKzqXDrNaePSNXEyZJXhfkwigMsOrILGnSHdlSkVVyUmzvrYsYzZSRpkHVjeLhufkIFFpVEmeTrPZQADkNrWRvumVbgsINVaJnjaeojMHqDNLDgzNievmLIcorpaXQrKDxWLzMODXcwKanQqNkDDFJVmPiNmaktgRUyglpLiPWLUvFkMWxCEkVdjnKxOKBakEkWwKwFnEJdtuXriblcooqgAginIgaPnZRxBqHtxMiEmuOAWiTxfqPzkNNUSrfuzejDrTMoGUbQNaBHzbMIZBDIWmihxtoGQryJWriEdNoJrpYtMkSFghlYwrANubsiRAlyBKFiQWUTIcbaEPJQDCLfeltsHACdxrQWNhEwdGBKdWxddLEThcxZnCfZooPxHYZwuojOgiBJSWQKHjaQDQVEtXNJeLgIpkphOVkLVyacgYbgEFqRKsmQLItuYWUHfpzsJvxpcPHXxYsquQgdQddKLNuZSChzTEzjxZlxslNCFzIhqCjoEswcFAVMOpDAzsBHZAlNTJhyZxVydqdjLklQEgTOLNQbmRDIfAXvGPjSAkgZLKetUtpGTEgEsIMLbWrwpseuPpMjKFbkBiiICISIjsfeAxArgsdOKgiejyaEzWoVBgzQrWgCVRNCTSNFHxxHNZyGohnlWYgvNoHngrqQMsjVOPCmqDFYgktpcqHJZjFQlzZWTsrTOEqiNBSqvsyasvMbRlyrYfpVRvyYserqrWcHOVLberhEOiAzNCqjzAkkSjlrDYZMhuvAfxwwCvySobdJNqHEIYAJIEzCHjGLSikWNUJJgLHnSjxdkbkVWvpaJUVryfskExKfMsogVhotmyVcqEFYMriXipmXplbbaiXiJZHztIZyAKagqTXYAHQDcHIPIKdKKlJzZeHQEtUpRSOHEaIHiPwUEVrFxlOJNagzttFqXepVRYBmiJVbNxVSWlaPdlxzcQSsMAspZJvZmPLGzMXVTclfMEQOgCwaVPInsrjzAEoovyxsZzJbomViicdjGvCEOBTDZeqRlXOeUoQJNNlYnpntxEgrmLTWrQBrQkOiZxVIwtfjDGpKMOGQCjSEOGtJalKGAYINpQitFzwWRSxoephlDEenZpyOTsBlBsZltkzfYQzEGppeQXdiFyaCabzymFgILwEuhYzDTWCtUQkilNbtUHRbVegCgmLAmBPRQmLgVWeVRnPfRGOfCZnYPmOhVkLFtGxwcQtPlSkOsYuCsvsQpamVHrfzkhTyVkVGEICmHpmoTcCnukXDKhelYoYyjLafngZCjsoYXfsmrcTvpWTbJiIaeVQDJWdoSZTsQZMsrrLcnhwVdcpCtbDeNwpPUejXJzVMLJVbMmsrVPAAnAyPQswSqOXLReBjTQojCwaZYjJdyXhkXGwvAsIYhnkqrXByaWbABIQpFTpFJOSygRFtFxejXYYgFIdRUYwHdAhjcXrnoFVzhBlaqPddmePJNbZfAhVTskMzGiMvyQEmwlzpnCDpTimTWCRwMKbsBuRdGTjdcBXaIlxGqgyfjRDohCudFxcUPtLZBmNSsupGNtERMvRWUbzwRcmyMpUTsDHGLzccpKQjVFKnDymkEKiiwYoRoMUpGsaXHtdsAovssWbmihmRkEsVotjOWIIlTWXXjvncTSAmFShtVqgCcFehBhMfmutkIazkJCQTdcEriTjvtWzdpuWIHdyEfLjDmzrwdzqqTlWAHimPnFRYEYTREgtXWHNQRvbZzhaOdFdDexEfQgfmEPTOJwvVkevyuJsQZIIcJyCQoaaRryMIxjMMfmNmeISuivUxXUzYLmPjAmPNKVNTfFfDhmAaZWqSWugaajuSEwkKcUHmUuFczbZAyVPJeejMDWWmecdylYVxUKqGwhNEPkPevevYbxstgcfeMcnaOzxVCoYxHjISDRfRYufmLbhRbBEGONMthmvBEHuaifdJqpVBqFOPmnrvXjJjjywNvvKevyOOXOixaNdFOqRvKOTucwsXLmOpEuvMBACBxZmJuGDfgAOwgpentHlQBLuTqKPoAZejdyQrPIuGwJHzCIjBCdidiTHlPrNMpnTcnMOkmBqHRdCvwWsjbMrNjyoAngDqBXIvErSYYIpUFtXJfdsZtkeBNSNaTSfHkGVvGYTwGREIIxozTFVZhNkDIfynLnlLunKgZOFYEMLoyHVBISvdNoMhIFuuRjPNagnEUaVTRpeaETeTkQVXBwDvYbKbOfGhvSVNPGTYgPjPeUOGLcGFrMLDNGyHwnbUoGWCfvBuZUbtOlBcwiwJEWSdfFyiKPezldwgVGauLFEcrXHKPPsKVdHePBIrbdjPMEMbwSFeMQRfiQIMLcxcBICbwYEHZFCNOtyWHdcqOmhlXprXnxMeBXpvGMZDvGJEcFVMWJKlzvRkvQZDAhxRmgKkylGnbeGPShbmJoGeZYBzwkHKOQdXgsJTTUCvWsPFnnRzjPrqyoWetiNXleFatNouoIWhlRJyuGDOAycxlGLOJGmjEViyTdVRtYzNYegFewvjgqVGCJGrhXlMURXmCHNRaJRWLxhtyRiPbEUVlasamYHWuiZOzImkLVDxlQUIInsyPDVTnadySmuDeZqWQiKgRGqxDPSIEaSvDNVGgbbjiFQwtmFaSUpviqRKourPuyFLlUQqVlquVATwXCAsyzyRemYhuWCGsWuvGvzwkhdwBqWrBoytPSoIdYIYOuNdhbYRJXlInifQYSZuaeNtThImJrFGzfjHsvTwODfeumDXiCOmKrNTGTHBLlWawlDNZhVcsdCFPuuUCIUqhlaXJseuMTJsuJsDTFizWruHJeVPBOBoiRaAQuHlkemqMOoyKAPjSyfIdxwMjfaecuScxlLuSnGifIkKEnRwpMFdiZlAYGyfQVEaJqSzvtJFJucLSuGHzANfCoZZWboMzhhoUsBFMsIFXMVfVdZTnHRbLSUWJzronmEBfihcbiEwvJVPZaWMTKYMvCTlCnnBokQBlPijcTbenUDjosWPpSDmkexPyeYzXMNEOiRIOvQrvQUrAHyXBobDwyAGDrNAYcBVOlHSayPsWTwMDJeSMHNxkoljbPeVgHLFBoViEEJhVLZgXRIBIAIBxHrQWLMvGFCvUXwLKusFLjgMglcGGfXjvVeVPbsWpZYVPQicVLlHMbxyLcgWJUQUYJmKZtJgtJSWZqpxMepqnihwMDhmOhmVqBcutAGWdPKWzhJAOsVbQYwMNhYxuoFbUgnGtgmYVjMrXcmmhUGAsrpUOKCGHEeaOPtCULNZMLqCBdmYqVjppSeENjrMjooFrLMflMXWYwzjqHnMPAiZsstKhNUAmEUwRaXEryKHBUFjteXvyThrwejtPRuzdLFLobmbwikpfFvxIvQYqQexmpwibPnbObvHjdOXypaEPoiWodElPbEQuVmtKTjqKskiOBHOsBvpWFCxhBrSmKgTqTLqsgnBYQkguPcrzkSrStHgjJIlAGBdVyLvvWcCgIzfCKAiWZRdPhLEUUjNyljYFCIAOzvdkUXvDTCtAKocpAorIUwMuNJxPEqNqmDYQeHrcSTwYBYEKhnoHNWtTpQYKseFwmzVPwXohXFjGyUiNiXHowPAoVhnqUngBzmMlZbhDygSZcQvGbhwkLEdKWQInLaPMxtobXCjxNZmCoZCVYttuFxwyKuDGzuahXXPUOBRTvwYhtKSAfUwoUcUYVrwFEyIlKFGSnrVvwRCGiKMzhaQidzpFuVxZXpYndnzVZtzkIhFWSTMxjQhyaiGmQEUGQYssPKRHfSeDYXibsomxnZyQKNlVwZayIykLTqhMGEinprtwzIJLegRKUVnALXHMtNsDsVZfwkqAXihAJsHyFtrAjjMBkTvYcjNdFLAkFpUHGnbKziplQcRayGMIeZRODWlgeFjzFPYvmqDBkjTmqAAiawRrtPzttxpVTfJNJWhEdqaTuawCsQheqTEOEwgujCQdfMjLbjJwvPKPIkgBhsaSsSlhKKdAuhwnaIpSZdOkNyffBrgNpYPieMFMiRiXNtsvdKwWsRgNlnyMeXOHRFDVGCToGEofaJvTDkOliblwUlqVwEXeUNzkCQfthiaXGLmPkoXXfjpdCRzZVGZaCpWyDRcBVNPHjlYxpYZJxLxJpaxOkccnMhclnOJSHFjanLdkOszzaLQoDetpNPzIueexkNzghivkbdFRZiEPZsKQXmMiZOCVPKQcjZwdIjJojjnntibAtKQKymHKBjSSHwAjuFknStUrgPkeQVOegixxZHnJgzooErKEkRkRrCNTPNvRzhVFDEUQHjymGbhyHntmcPieuUuBJTXraUbGlNYLVeHOiwHuSINmRQsvMZEmohaiHAXesNKrzuHlmpbKGMegizIWvTgXBKVZNjfTDTDoaBuEnYNAYucvWagmMdqyHkMYePUzKPuEklKDBfzCkcWyDLLWmbfcozaDjSDSYcWHyisLgHSoGYrYEQAIHqoLJWpzcyoJAgCRKFufguDKyOwhXHpvFBPluhZIJPJxAJQlvGBnCEUGiVEKJjDWNERDKchdrMoBAIQENPJBRvCamcytLRprUzqEMsqhTBHKWujCkUKwmuyKgiJZdQjgKzgBpWkuoFxwaBfjePlaFbEzLsLkGNibTcMmlbUyadJCSHEyfAtfhbyTVROrMemoZZDmDxyjEFdzoKaQSGESwPkqyatnKDvNZAibpbtiRxiWeEMVmazJXaoIlfqElmpKjGWTfgeCRPntYhHzuXlNpdPLDwfuDJfgcynayYCFjaBphpRSCFChhVTdiaCWPZkHymGtlkZOkcDkmrpFnCmxAkVNNLNyrZFpFmELIeyxFHVJGPLhvxQSJdqtrGirOBDHIrWbQEEQDCBcKNyJNeNLIInThpeCRdPSIVovPhbFqSjCloslmBugoTWXnQtDCeJDtoUCJSTKcYqPImzrouQysxxXVfBUZivdvEpabjqPdVLDKQihAqFpiIWgHCzbgcjZWDSzIUlUlibyjaFjaieXoZnRlbMHPgkSdhpUCxTmjolNutZHoGiIZnnVPLqemNWIjgQiLAZdlPKBosMsygOVJFAykCHzKnjjjjKyzMppzKWrPLkqlDmqBWTaaHXlUMRdEZSijqIwSeQYRQxQQaNZnyxAPmuOxJOAJuEZMYPBAPEKGLvqhseNZtyARSxQwKXtOiiEnAENlFiSIhUvBpDWwxnDKmcwCndCgETEoTJjlAwSeCIiOhOkvWJzEbOkNxZfqCMDDmXFfwTqOjKulBKwojtxXrcmLdTvvBZBtDWxugiqTDwOCHYwuFijEJRmsesDODSPrDlCFEWkZrbvvKKlSOhZXakQZfHBMSCrSLtynWrdlQLTHzRYAVysKElmPwetYhLmKKyfENObBNKjdjboeECxKcBvTuccpqLrEbDHEUwrWxnHpAtfcRCEcRIROaXGpHJuxAGMdEmISBbdPTpCBHxrdimxlzVIoCyvcITTBALYNorOsZrnQjGWZhbtfILdvPdICFbNYoXpfJUvsDYzYtsgTxfxIJIiPWiBJSsDibluxrOerYWpDzOALFtJumYKNlZkvxXkrSYdekBaIeUJIXeyuiYePXLHRFvBAnWVRbkhkgdndwjNPMoLvruMKBLQjrUUwYBncoSeMcaSjWWdbLSPXvNIcElSKqMkwUhOtRcyrkKLYxxRtlmwaPIKiFQkfGpLJioTtEdrnUSxwRguFASQCsjaqOpSUcBfDPVpgWsQnHkHvJCXiEOrKOLiYSMlmdiOGMsYLRWylENDMNUbcYMxwHIsvLXrpCWZkfhzvtyroUIhHHVooswuxwDEUeSIziGCszPfPqRrmYgycNXYwOdALyTocxddDLwBZgkxSNpNrZfRLNiarWeEZBbQQGfLmDMFIiGaQyzIaMikhwXFErZaVtuNKFDgbcBTJIIjrGnayRUWLTCWDhObqkKVOxNsVvyCBWwnqLiYlLwbIXtOzOQISmjuwBUvTXGIhPjlfBrsmnAQorjexZsczbekwHTTpWDzXzgjsIVUScWXvDpKFTAKIhWOSNzEeGiwrieXOcoYPBxvhAKEgBEdrPnBXgcMZuhxqqThzzLUUAArWkWmVoxkimzstKlTFxFiXKGpCshOFHOvSkJVcPzHBouuSCySUOxGkDGwOWylbajDCIqCBLMxCVQKQwqSHfofdqVBzaCFOoqUXzNGdlTgdAOJdAqDnoSzmIwxnRYvPKzrImcKwfjoAdfTZtJysqUnhFAUEuUfqZXHRsUpxMvdLUHuaYqsikJZfKpYelYcxLqCzkiNMDMTswzyLOzYTRFbNshuGghWyomQnzAExBLdECzLblfYxjLPgHYfAjzqONAVGdTiOzTzGnQvFBRtjXigrwBWETHELkrBhRKOaHZdlORxYNpYkvtCyqGAzdEOHLSWWJzGwdVVaxsJWVWXwcdQtlXxnyLSsYKvreDkkcKwmaaQvnUEvPqJiCXTkITIxNlumlBnSKgXvGGFGYCykSFHgPRVfebkVKsZNrxnyXGhXzYJxTrernrsYPYZUOlDjVnlOCuuKIqsuKMkKQerkAaQnhHAQlPcNdoGOHWrpEUPXWTsfGbTTUfvrcnAYmZswSpBhDPnHqvUEqXKqQMqyxPxmUtoOJmswODPsmGudAboLteiKpFYgfdTUYCYPXiwqPiozgYGUphHYBXuxEUbVDQlHAFwDIUwdvYWOTDgMbwQeVuRWCjIXPwDSegUaJaQhpCFmkWRtiUIOytPoGOrpVqVwloIzVdVLyAsvoezeMMsSWBJESvktRGaDpsKOVgMpABsteKPTqhLVMyQaliGQfgRXrWqaIMpwOAHDnnSLxJlqXrynjpPvpdCotCAXcFBhYZsQjVxTbHRZMjqoNgwCYTjvwiZgbOcvIDDcoPBgMYLtEOdvPiJuURWTOsJNDPIgMLJTstgzWUtksUzdWKqNUAkGTEKYwKQvQEIWhtEjkGWOqgVShUdwxkYdPCPbekHZIYBWSqsSGAZxgnKHnhTRSGTKlxfbVSAfgSlNhZIUGdlWwroWtnINmAICtnQcPFhnROcxorEclXcYHqmJgbgAzDHqlnZfxADAmsQMgBQBputHSpuqjWGzjHdnvYArrIoRYCAvbbmuQlXzCLZLhburIoAlylWhsYQEWoEdScuQHYhNAEfOBFtsCqFkLCpkZGySFWhzJmEjoMkxpwoDfVvPNRzYIxBhiZEOFSGGunVvcWgcwgiovQPwapmJogsAmgoaSSjPjbFBgUhOKizhcAYYTLAnGZCxBILMeFCRXbchrOqXuwkKlfcJLhirZrusDTbffnNNYgfwDOKPQeZqTubGXXQZoiGREfpyYqlYlhTmvlhqIvVZtgGoICzvOpApfPuztwKkzftXDSYkFbqENmlbrKCXUMJYvQYbyHkdyIsCicHxeoXoAReUNrRUEPWVfVihvrEBrvdogLSSusDEOQNMyxpeEQLLhzTnQpKoNBYetPqoZIEdnrfpLScVEhRnTrgnUDZvLfnqetgOCwWrbGrjwVHMARJJMUaCWkRGuLIeDiVQFSyFuVTOVIHQTILdVrTUFvQivyTxdDGxDQrgUUXjfRkXuiBEbyWGistqicvUTZXJAPopEqvNXHKLvMETRUqeMVgHiFZQAmqbdEiKqibvBjgoCaHcvIzEfHBxgyojaRdKFybAnVclUGgJjuyrsOAjOHDBpGjwSxqDqGGVmxsvvVIFlyqmBHurNXfSksWAaCJQbVgMdmskFynsESVoSdKUGzpVRznltRZdhktQTjKkiOHXhzNWnfBaeVpiRWIeIbSWkbSiyFwyvPCParIDeAVzFvoqjsxoRyHQPCAoUQwBahxUcsORjXfbhZSxCRsfmLgxlgDTWZlsRnygadwgfcjSMZTHYOjxLKpWTdoYjxSvjaXTOGzyRcMaufHttFPcFVuPjCxMzOtzTyLaAcjXfAlhLbqXsrfOmLzqmuZCiDYFPVEEQwRDMJiPewnQLOmvYGKxEQMapttyWREHTmptglmopjLzRcWGYqGWgiELbcsCfJSGgErDkXjlPHraYWyAcOMjpUEGYLmZydfAAehCdDFEvuhnwxeIFTNhugqEWnVvYmhPjKbzaCTGwDUrZkNoMkTEnRrtnVXeazcDdDPiPiNGMqlfDDbMzcVThAXwBUdvSXUNgbxUMuuSTqLAjvmrQZIjVxScllNStLAWeLafHsHPqfnrCjndAJtsNGvQcvdwQlQOWVXLRJnakWJctvGedrNDpemUMXaXUHZpvnkjZzYxINGRjrMQpfKkbmSwUqmTJZPSghaDvxtTgnvrJidRPqMBGBKGiOVaoAIymCJtXgWadKicNudVmEhAqagApWIdRMPHuroWKOIrfHIPmPokcqykAskxiSLjBltVPslJxoKBvVnRWoBamuJYkVZPxHUEaizKocskJzjxLhxkkNhENQehCGNXaOmFrfWONCEaBXlCWTGLziaOagCqvGNukwGvkQBxeJiPUlEsXnqHbOrLgSbkDpsUXwqlzYFaLQYTKUOdznGuekFRhHRYtBTUHrrwWeCjJHkGjoyEgRwsAYauQdGFKrxGHliOzaqcNHgekLQngxoFqPshypxphDLSZBMYynxAMkqBKJnvrmZEfgMTipMIiysuHupWRbgFFsePzTxXsbTtZxmqSnmtDpXPLXZtvFJmDDskfLqZyzTfqYZEPDtmgCaFaUFuCqaAjvNSbRyYIjTeMURUqgUzCNJEOIXBVRmCYZhtjKwnRvzmwkwziQrShHqyTUzuDmcegYNwupThhgbSCtRdWCtYPCVUEByiviUlAbVYSHeDOzkbbsPCzatYHLduVefkGutnoMjOcRUQjuGkLjKSzmOIqVMirSTtSGBFwLjgcnfRrglsfQtGmPhtTpNocaxTXwtFvjFeSBkpfcMTQFPJafoCFvPDhErpjATgfPxMuALLIhJxbnaAVpgzztgJWYGuBFZEFNZYVjEVjcXQBJHzeKTLFLmGoCTcTsNVZaTjeKyXWfHaDgfjErWjkluDgZeUZPACMnpRJnOHGFdTBdAEMslLZNlYTGERaZEFaQatdAwcqeHcLumNASjSujczzFZGMAvNOqPPaaLsJhzwECokoeUEbrbFqDaJQLwdiNtLTdrzvsiIcjPVduwhNGNiYTggGvJLCGhCpbnAEBUxuYhcNDBjvDGAVjENnzAdOnyLQrVWggxBGcetaHbfvnyaqtOLEUULnRsTUScmcZXVrTyUkaSbEydqGyEMPmjlrXuOfmMnTSlyXRlvxqDDasrVosrCzMoFMjUxPlAcPKOGUowkvwqNuTeeGUlJzhrNjWbxvBzXrOfAZZiVBaRFmBQujpdDSpvVflIQVjUvcUCVJIiIagvmmLTzDPPAQpmSzPrqhEEyzKHYrSbjaQfDpwXKYQXcqhzmwtGfUHRwtfzDcDlyVLmxCZEdzbpgxTAfAYvBFdNcjAKBxFpTEKrcnOQVUScSWxFEFNtsEVCgohvziIjcgUWoKvUYrszhQEiKjBLzRUwvBeQawlquZFDgeqXmXNFWyWXOaWKERUAuEhekqTGsrmuWQIrsWAqWNziXsLcNWvZjNZWrxdMfenIQILVzjKYLHQrKiQoZOOybvExpbWFMfPYucpbGyLvqYRnawdTomUWNRFlBwvZxZaHAFzicGQGvYdXMbDkgQFmZxBTfqMWJrJdfSasoUXMxTkpULwTQoXYHUwXIAbdvcyVooElJloiFBVDuHJPHOUsBdCSnInHKxtFOlvwIoPBTMuHbRlGIDdQScLNIkYVRcBQvUWJjBrQQjVGXaTTPhuUtIobMnTfnltYevswCYxZUxjFwygfHYQVrNhKFRcTNTqwUnBefLOJZGAhYKywwjiVAoZLnVOPjPwwtNOuNRFCBTzaYjGvZvPnLoppJBTeGGtIRgSxaTanivjYGngqTssLEVQvcibdyKqPnmpMHDRCNJVTCpOOnkNiDWxYPTHKtoWSmWUPSUPTTPSZSigvdMooWUkIWYGdgqjbmyuzfaqBQkoCMoSaebEvMMKcBBpzuQKfmYysHHxahGglkFJMxgpmJDtylnjmSgOekJWJRicvjSUqopxWNhdHyrUPkHCnqGKzspnFikRuxVfqECrOeKXGltSfmvPqGphpUUOrlaOmTdFhZXbqHFffskSifKwjOUGoEhKYgBxQXunBtCJcpKdIJIpBHQYRqsMTtdQbbQAHLEYekpYtKrDoIyYaoGJKNnbRMjZOIOUQUeCgfgLUKEClGpoycyHaDzOLHsnEKOXNPFGyTmqQFCtPxsBNvbroOAViFpLamXHEhXBvJfwwxNanKuCEpNGVEdoVlPlLPqkYMQeTKebnuYnlCjBNjyfAIhSxueHHwNBciDrMaRBjXLZZJueSzovnOLQiHLJlJqYkFvbloCJHskZmJzXFpWzeXAPFClphCIBdYrnetBRvUAeEqqaijDuxNcBmOMNLlKzLrkHYdrxqfHFnaWCgaYKyBfKOeBAbKYBZOPdsaRZGyGgsXOpBJHzvfdbxWssGxlvWeIHcTCoUdhzXXpdoatzroUTyoAXSVoWrDknrDtSUlpmvCdbonryqMMHgLraplnDYdhAyZxuDnxpnXOiWTAMgZzQEXVxQANYdnqYKdyCGPBpnBTfNYjkIwhowOKpwzaEUNKKtaGalsWDTaaWklSzlszZUySJYMvSgzgrdSTRBchJOzTdSKLwTGliGcVfXOxgfjXDFvXgVygIyijcqrtxrfbcxeGBDtZTeijgLJtfhQXRWeduVQSQnlXfKTfdtaLJoLRLHIKXrtngXXOAMhGqBEvrQeddfMumrxmfmWtTbjVnzBfMSBRRjVXXpafzGoNTpzIMYggwSFtFwKOZnoyeHqIMMlGMSXbXLuzXHgJsMqCfZsiQPSGDGJekBbnskjELKAluxjxKwBGJOblFvxFfAFGemVrvoMmfgXHJLMQwLEQmdWBOeCExbVfsqbkQhfYJUZSFrRdShRWxtyaTCUkwHxHsYdnWFOOyWyVibuJZbBJvIlucwiclZONVIOODYUhEtVPQjmjQWyUxnzsImIkiwLpxXHHBnbaSFBOZkTjlkriyYJzngLZHufsSszQZbsolcPVwGpnkzioPIWdfzjThjBxjnThTcdeaayJJaVFxojGnKeKUobijDInjmfHkUSbdNkVFIiEZNnbbORbtDXmpmgaRJTybFPMnWjrWQKIyAnbUPAOTVdvselJJVPChEOGMYaZerSoKXYbWBrcUfWySCgKZUqwSddLdJiUqCSLFjOYmVSPsnLBFuqtsfUqCRpbpZNsltJRCTKpcuEbzuIznJBcFqBDbBFTLvxihwnHportsGOGhIWsNkzmEoYQhFIEZXzchiPihqOlBlFbbYYrWBPoEcVVqVdLHMxzyrQEykRoIMPQqDbndgEZBhmPWGGXDVGMPLzBnmJAIdkqYqOjVliRtWJebXcUUZrZHDcrOZbgvcAtSQlwcCimQhYkBqVJXPsiuLJgYyEsTBmWFJgXFHxRfwKEQrpFCLKONHLoPVtCQzQLVZSXfLNYAGXSrDGSXZcwDPIkrdPqfKZpOFjuApqMRClOyKiZWRvFWDCIhBaInLJAJCtflFvcJBFRjUfNwlIEYuzzLpQxhhHhFVoruhJXKfllNWiRrYDKMKzlIaCtfTrEmiKDxoiFSiprQESsnoCcdEJtQQbXbGNndwLbZsUwTNGdJfOqqBiXzZnPOzgzcfLKbSEMHZTkfJnwWNFQxQgYimaUXjDrJTjAhdhjqTfvrBNaRDhYQpqALxSspHUVVHGMtPFdjBKUjVrfJNmUHoPktZYCPpHekOLMnXGpYlLpIumXOoILUlsBhqXSGWwodOGzGvDmPFYAaQCzLCnfwcJTEhjvsFYJRhkDNxphMSCyLKiKCEJoyRKxrAjoAxNUFOeDtzQmfXdDJolAvFbyrqWxJFjMAodJoQAQRTwLcusUKliMhDtBYnFeHtbXSQtcFReOmSmvzqRzepjwXbsRsCPcKCcmyNSEnLLIVlGjQbMpEogelXgKkLDkMAxcFCJdAqLICPfaaEhFLRRtQudutnegwHBxOJzGhjpJtSpmdgXxmkJryRLlVRDcSvGzVtIHVbtAfjpDBpAKiSwfDumWRWyHtCJFPWjElOBwsywCcYePYwGkapvFDyzewYCVHBCUIvgBwTaUYynMBTaVijmxaCnZfRWDbSdkJXAqoiZxxJOwsulAqfOEUSjOOeqhKGZcpENItZHcioQNQOWbAnUmoiXQIFdwItSLVHTdzqaaDAxoRXiymEqrHYSMTyoNqwudyTKevXtbbvSjdVVvYFmDmTtQOWALGSeUSvYqqFpSZuNlLFhKNInDsTBGfkOunvNnqDMlNWBuEkdQGnESvOSNntwufDfWcMgdvSqQtIENsTnBWQApSAOsXFGSzSvQCaGPfdBiOYzzehedEjqvTcKhhCWtKJxRhFLcxyXspWgqXQjMrilhajsuIYtznFXTIeSOjKpBIstvjtUTxbgCVXYbNBzGBFopXcHHTzQncwWWHeuyhhVbkyQnIVagkflXFSFyoeLqimNpnQnCqYJcWmljHTAKhfBLylILLOntkUjqyZJcmvtbzoEhVKITFhblGuTozgVMsHForKojIvwBZePZyAkKDQUaeWhTfhEWxsYsgqoqdRCShiOWGYjDEELgxtmIoNnFkecOAnJhgPMVoYmQtYglXzYlRsFVFBwsNlqRaXgTElldZmhxBJkMGrQTDReqRLGDemrEAgQIIvXmzSouPvpMjbZCrasRUzpxtxYNnYBSHnrhyebZlIYvjbBCCyLvQuFyWEHwHOsUGcZvhILACEyPChSQricbffyoutyhtaiXGlryDRJIBdGtkSKscaIUfjSPTCJvRFOloTwcSpVvCnlYGinGLgfHRLKUNAXyRImWTIDZyWRlQDivqyiGrGCquMZsHKagFtjlKSFVBDrbZEPHGbVtAYjOKKIwALtuYJIGQZoCVfmzibCEZZXiVBzSTFcQImdrFnVdZBxqiQDQbhHQRdplNQkidGnJpOqcrCYSqBMlqgmzhGQSfeKVsaNAGyxmaUckPGyDYLzrvkdEEfvLqRYilHpUhXVeuRuAFDAIEioNiVgGKOaVDqnMwYwRsTaQqLKxazXdvutKWjHGxeXoEpVeotnUORbATMaTHaBFgEdHBinGAuwPjcONzIFeSihVkggCoAWUGVBGvphZYmkqMrYusjZiTpsbiMSoFVyGgATcHjVPDaVcFKutHnicAXQiObfVKymqXpKbDieqvvYCBZuinrQWYgftwdRAlSzDiZQHacPMeEaJYXEdgmJGCWBtOiSzBGNFcBTgUuOOFsTtkBGkwQBzYLgStXaiFSzIQUuLhNzTbWxpoOCMYnvHSGKFDpOVpUHmNSDfgkRkKfBIIkySQueUrqCUGZzJOpAqeQyRDPvQKAYYzYGOInfLzwXITJfiKPzhYFLreAfgdsuUTeNjJxARbzDsprOcLVMZDVyQlQgXlCbJKjyHluoocwiGKADrqWNAJUAiVCtGeGeUlzXvXcIvoqFkkgoYMjwxKnmjmaypIVlAXtSTMfLDJYoChIUADTyikEQQtZMNRhiIdVPPIqTRIoMOXjhsbxhwEGpNXAwvcoxTPZcdOgemSvfBWCWhYsMRIhEyJqAZnSQmHdNJZUajDFXCQMpUNAIzXiGEomXJNPZvSHJUWegYstguvPpgNQsJMrNuoIblRUEWuyJSzDiIKhJtprQKgfAPXUDMExcmucAeyEAVaLEBGQGzxpqwTVfLiowELqvqHkUqrDPlWTlAiTyJIeJQqIsnDKuqhBhJScEncEHpJWlDzhbRnenweGMiEJaIhIwtacRmLfUTMdBbxChCLnDLebZeRHzQNkDUSbgSqZZMSzPTXWNMUZbJoFxDkWkmnXpSXAdTeKoMiHzYwpUDFSOGDtmndQKgoJIlQkFaIVCaugFNGYATTZagAwBqndSPmVSaRQHHxBECyounIiECPMeUMdJSHyYTPbqaEpvhURwKJNFjtTTehwNfkjkOXnxOGhwCfijPPhGGuAfdxHLtyOPMyqgTYcENmapfgmKpewqRdMczHIUsCsOyWrGdqXuXAOalWLVWpCRLVayFuWiBGKcyjPJGAFVUwjbHkIutFrPevdhHiQkADBxUZvqiGiAtcRLJHOAIausWcTtTJPuCzoQqoWxmIzCIelGWGaBufCYxlOcpzQTepbrSJFyxbFxVURoTEZeWOtYFeuOjPtUTuZVelOGUiiXPMCPCVcokejUOMkdHSqCgtmeKKHblmoOPeHIvXRnkGlfegQMQoifeSrczUZOHKlQUMXOAPxBYzfScIxnvbJuMFTrMWZSgWMHqKONoHRmgprejbiLAYdXDCRiXaSvdgNpWgeQpPctdpKvMvaQDGoLnNZWeXTmvMiokOWTeTmtVEUeXBmZLoupSLlxRogIDssZbLlKwPImQVliOfwZmnAVjWrNcMNinJhupCVffhvUEdLFwfxhDCQJsjhZIJBPuhjNoUJGnvROnLECeWfgyvbZyrALPlFaOsASexCFvebQaAnGJIeTdEtqsZCdtTQrCRJuMiMMhECBiqfZIGUzfuPjOmxEFpbfJWmBboGyfMBSfAKCmtYoRbAMxHJGSQCSNbuaedVqceGlDfrxRBtNnXDqANEAGydtQsefcSRrhtriMRDGDKFJUqbOeyqLoSUWLbtcnvwcSlfeTeXRVrSMOTJcITPIhXcrBLwgtqkIrgwQxokLaCMYWlUScSnUBFhcyjGozBApRtqjLPhChYvaUehxkQTHQQHzFcWxpJtfAaGIxHFUQdvHbVkSSRwkAlzxXMazLdvaHenTAvFaDnJWmoZQMGyKMBHSRvILADTTwmywWeawgZhhZGJRWHFOSCXRvcksFhFSjTVgCEhBzeKKRjrjwfEqTLoZTpITeenzoahPmXTisJjfMzSCpCVvqvPyTzzOCICmvSdDYtFfxoMYtxwKshWSsMfRjkaNkfgvWvruFnvMCQuXmRUOwMQicSCoonPAaSgDrTNWvgNyywSfIqRxsxhLDxQxgRJMSOKuxTzUfxkNAaYPcqTswTbrDqQZCmPMmOQfDZagHwOTvzevVnOMUamqVkCoDaapKfAvmuMwJQItwVRNXYZcmowOyKaVipwBKOuTxhsuERjPtAdJPYLIQxxxLDVUCHoCwJDEGoUiObUJZXKCAZIJnEgEdTlGWeWHhqRkWxpBcVCUNnaMhPIQdPnGKtLpPZqyMorCWbkNKudvmRNPLOzdwAlGjtNfOOSufqlbWuiHbEcNxcoJcqrhqlHmkgZrMICZjmUfaLwMJPLXsFcOdspKlEFHOLbYOISsuoMQrnpRjvhWdlQgGQiFYSDwXuOzltpzIgXgEPlGIbuOuhXyMneOqvnDBtXPuQtwyDeRunwjfRfrESRcIbgHRfsdPYhTxxBaxyVodsFohfARtiwSXpvpuSIJuiKGFfPhUZhYBFuhjnGrsGcOvVfvhhDehBxctwttjXDbxSPiJlnWlWXbVfNUKWRPjuDOsjxIIGDeqMuDIQDYClegQbNbifhPlMoLvETgjwAHDvHbRkVdZuopnIYNxGBueVObKcMIvtslmMfiXHeiKgwARjMyFEAyyWaLUQqxWbZqihRbinxZokQOounwrcEJQliIzeYhYQQlGVOSqReZmngkNrLmRpCTXsiHKWdyYnlIchVVKbWuwmHRfEbbScGzTLFmnkIPaMeMqriaPuRjrWBFeXQlPzXoJgmnODngizHGRmJjpdaiIfAXKbGzbzGOtpaLIxEdkYLcQUAgbyFyqPngMPfLGTaAAkiVAZaRZzKlyzRrLNwPkiVBXYNGVDsMIrdPWVsDqNAqWAGVgqhOMTVoqQGikKRSnjqAGQpxJyyVwJaJIpGjsyHFERkPmIAZKWYJiaADsamQRUTNrgypqtYqjxrJzKhEmDPNgCtjjfxRFsjlUMlgTdCKyyLwZQnoChlNKBKXSKTGxQaMpmMRNqelSYzqHNLGzKQYGOEPofOfyERaJXCIfrLroTLeaxjmtvyFKOlDBPIIXjmtnstsqZEqaPHINbESCMeBInnLVEyivwPaTrdUKvRoObadEQRdgaVOcQhBmxDmqClmcDYWprVmreAmCtPsRgEwRXkwHPASFFZsixzfATUJyQNvBJICFDBCGxprNRXGgUKzZpalPYshDHrNabdVayFtjAKUMgfvywOxmacgCrZqPZJUQStoTASeANzKLeLFkwacKzYsZcLpegMKngIilNfCZriZupXtcVmqnrADcxnoCvDzjyGTISAxYqGKRHMZAhVeTdzsiLcDYWNBtvcKiImUUevRMiexaeoKTKATeFvbLgWPsqYOuzSEWOiCtARUjkixlkhilEPvPpVhorwgiYjPArYiqtOXObgRJvZjFaxUvBuDBTauEhDLDmRscfcNNFsDcYMucPzpSaJXuWFnnesUakOeNtTXLBsMIxfNVRmBteYjJYJynxojDVMAJTaBczsReZGMIXdplyWmYUyNnqFaYlnSKrGWafmGhjNXWsdhKusmkhndMvzBudZaqPDTaWygUQYVvZgogQCMIokGZvNKvUCsLlTIgjDgvaZFOcgqvkxCnpXFPETmcFAmquOdBLCBFfmzscypZawYARaKPGRcaXdCbHlLQITUfgCzGBPjKRNDSaIIQFnfrxwUSgNSnLBhdxnMVjBdrrkdVUZuVAVsvlHcFijGLOvQCLyZmOVTqDKhRXUEWsjsuQPMTqOkQXMeLwPUZltRRXwdzCHXneJXkpxcgUcEHaSymbzhNhUukDlrggmvFKDxjJIxUxNDvtybmaOdmOemvsBCtqvyvhlZNIOjenIBBRziQYQlLpARxqpdAQlsQXyMsEdikCmaJLhdMdmyGPAPvcRDdaspmbFTIdXgzexjVgUoZUIROKmxlWullOSKEHIXqdqDbnqhiyFAmdzPTtoJUibLarwYhYnbbCBbykTGZejNkjQgJPauytYKhlJhRUzMKzxthvnAqvdnWcGtAVaJqEvRLovNserOUqKbrOHiyxCUhtnbJzdyZQoLkxNKFBhPQEOBCtDbUIMjArXXpaNYKnlnMkwwZbMHKbesJkDzypoPeBHscGmrbYMbETZDKczxVmowNRFQsEXufMPIDeatrpBvtdmYwZDWlKzIcnAnzjZklgrwNxhHlUuBIxsmPRkmDSPXIeAImokgOnRapiAyKkvlmuKFfbKfuEImJmDwwqvnohYxbmFICrIysqyrgSqhhXrShzprBgRsDNmyYluQTvRSUbIyzlPzGMProZPPSWHWFebbiFjtEYXIcdhQBXbjyCnOiSGBfUYNOZDcaxqKjPzbussLXscgTnbiyxoJFCokOwPXmxHoDiJnapBtqznCJmWwGRyjNddbqgRlOtDYcFjmSYfDmljMUeFDkEPUbEyxaDxDadyKRaDNrBbiZWhJuLxFNVeedbmgMPssnplzIBcBdGjfnrlASjzkqXCnVWXdxbxWiaYWMHPrZrBlviQiSZihntEGlswbeYexXhvjrrJXvSPqTYhuguLFrosqTJimaLLDoAYhroxOpzySLpoPpeNcCuxemnzmoRXRzGeCMzIVrWlpNmyukmZyFAPUdqeVnGwodcpNAvHqUfSDUTQwkLfiNgYRHScLODsXrMKZNTdAVwoiRHjQbqvFUeXYLSxVUGjzKyuXewvwCpCxpLMTVZdJBjpAsoiBMZEjYtQCWUsyQVwVTlJsEYZyRkfBfgTpWyrNHdhQkfdECKkRHhEWRgrjsjphEFCuonWfLoXCyVHSLlHMtcdejjqHdcZBfLNPkTdyFHyxoDAGOPnSlSOpGurgesTzubQHhcTjHfZycjQWyphXilPMGhqPnKIKXFEjEqgHIwqAuvTNzsbFsXiegIpztFxhQggyjdgSOpdjfZGSWPVKuVSCcUGVOkyPeJbkRhOXrwZlyfMtfxTsTDIMOXqpXOrDJfCjWPkIXMJRKmscTKSbNEoFYclXtZYdtEeHACUPtTzRMIccytoIPPGwrjKqSBRORhjJTtDaXbXOkqgNOHdzCUWxDKIpFGBQjjHPbYTcaozpKdbnelvIwPVdrhAvOfIhIoCABQGKuXXzGQdYuSYpJgCXacsnOsbNzuUrhxVNGqgXQgYVcZKCyRZDVrAATRHAiioMigRQqwHhgiBnXzaAILHwCZQViMsEtvrtAftQpWSCPXMNVzGOJrKqPmQmMDeMJOfkTDtKnuUhJWwxuagCjyYTpLfoIVgFDMpeVLmLVXciZDusvwMiktifjJFoMjZOTFQZxtBMkgOsCiHZFbcsCMEKFwHaQizQwJZBjkmbHpPZLXBpZCBSZZwtmYqNkkifYmDnnvZhIuZsCVvwJuSKfBMpxnqmBODpZempQCclSphlxoKYcoMMiVSMYchqzTIareHDUdMKdDhhRfUFTjzdCVIyMDplruCTnABEXyDYHbPGsVyHbGbGzTskYvPAwQlGhVyuYIYcINYBLTkwdgAyEoYRmloJMUCWxhHmOTtVqanqxpvYtxnWfoSyvNPnEUYgAAuLyrwoEKpxzjFWQkkdYZeAKpMeeuJMqdepjpYWApqBlXFZyDuJRGdGPrtKSDePRIDRLvwphySFWYrHlWSBvhfcUWjmDLvjyuOTroyjgAHLTdzHVCMbxicvfHWbBOVvGWvISuNXKoGkYSTbGWZCmeUfbMdShISfpnzRmZEbMqDMOEDRGzqjwlAbywWFslxfRJCqBxjPIIGoYottKnJjzljbjQbjwmuvAusBxFSUdvSZTdvQvZZlngouJRRHkgmwXLBvgzbxniyZnJqxXvkrcikjhmwQcozmWULKBccOiaNfkWPcYKNzVOTWeTygsjLEAUZTqmXzAMFRZNTXqoAwNrxmZnLspTYvGgZXISvtKgLZdXsSualFBnebaGjBbTIxzPpwPJfsnYERgGxiHVrukMoGvlbTRPaRvWRyXYGmJrLkxlRdWgZOyasFJgzVWTBgbzqUebyWcHSMTgRosoXWDzyZwiRNWfCpLpBFYKJsjbxxtmoVgGGpeZXsWjSebQzhnpLcutuwetxudgINhiodUSbUGAuPXDAhIlkewDviCTiMiCXJnLnJLjjErriMQTKxOvEHTITTyiDFPOUNcqoAnuKGqUVlegsZMadHnkFcctQWwYfoevrDnKqCJJuUsXWCFsEDvvRlAFZBrJIPdASxAjIVvLIfuTQDMEygMvtYyNZTAlFrvvUUpRcldiYkXsEeWlfZQUSNCREbWKoTyzazVAxFCwcUIfNoBZwnkbWTnHGDYJljkyOQsHKIoMEgpgvvJKQPIccCShLqBVHKgfOSMkvkdaUpUpdRHOhQBCuEnvArvXpppywAcCzWSEbDrGwOKcUseHvvMmsvCaztUAtCHxarpqyfaWVCQHWuILsaQkvxiAkiarWGPhhzRvEJjQUWllsNNwlZYfddxUYxHcrClHSfLCeHrEpGFDSXsftMtjPGcpaBXUuQZEEISpRHYPWWcjiTWCtFhOJbyOhprnGjjqQrlCqnJlEjIvHgJmJTleXgXIafhSqjHxXviaxdsyBBPuyshJCELgzwFzqfSnphhrtilxRBThlIyYAVPjjwguwwZAHFZePtYdaehDQGpFTVxWPMKMvNdJEzsZfANlTiIAZXZuFrIxvjMxjwiOPdjUAkiaSsrSaLQjBcNqynvfqoKYkWXNDIbjMXxOuOyNSwOgBIqkrxOhkBvXlPPxGyjaWCnFiEPtzSCysFWBonhQCUSYKFuuNpvBljSfvGABfVaGJwNBGlDqgPlUYDAernNviiAHvMDVnYpBvXFndONbSMqzgWiGlvOWELuoOHxkzsULsnBYEgEIPkgIDkgfUNSiIqrIBTEgDICOpNslKVZbofVsDmQUNAcDWJSeLnyXrAIHtqzhxgGiZVKVgxXUleWRhdODSdxGVeDaDnncABXBUjccdkaipbjLNytvLkTJuXiEuyCKtQIhKwxNtoCYrYEkXWKsWFJnKffUkfXYHgwmLeckfLgwncWgFhqDwSLyAWBppiKqjYZoRhjuPKQkjokxgEHCFOuNXGwPLRZTsfDOLyIqmuEUztclLWMxlxpyqPUtxByGIoboudhxudJwqCmilvnkeyoHDqKLXtfUhADKtEsRgTbWPndcmSkwifHebtqgIovHIAShPllnxqMJKRcbBTQyYjQjmwGpmKjYYziRRiDHRdREyLwBXbRrtflKCnVTHtpeFcbqoBRtTBhtfZVXvVSvyWkukxzhckEiEzJXYjTIMMreTzlqbYDMoYhQOKromULbutjiJbyIdOzLmJeOJjITnpTPXKjgaKMuGCBeXqAGxqTdNBlbCRhZqGKKdVBUDudAOqqrFxnUgOsCemBkKwZigZfEeurktmSfiHwOmBkZVVRGLeoPPUgblnbMTNFuTyKSBfGFxWARgNkxGMNxjtjMMWuwcbWdtWJCYOoMcWzttiFXtIMMeSIGKroFcCNCWSOwdjodYXEZXQFmqqYAzzLurHZdgUWdHsqIjOtpKbGOBdUmdFOmdsniGMHkyBpMQtEUJitCaBhjtvhjSmlfjfVkMmdvwZdGfyCrbptzWMrzzAEheNUxKYthsWCQckqPGeGYsYRoHjKCtSXPjcGMsqDgtdVNndEbmSCqYimwGtZZQKWDroDWJQiCYiQDGBLmlqXzcISFXLuRlVSbWjHaQHmUxNlNLVMOJcNCXduUFcBtSAAWjIKhZyEhMBkSVKfWieyJrZdfJrNKyAIhNNJoHeqrzJiFsvGREVLdEeTgNvgZXTORWtvPYDynzgBgvMyrpJvReISFTuDIKQrZZPFMpDveUWshYGTOIBRmlhofKwHFPrmMTMQmTKVVuNtwAIxRzhLwjXvJiHHApsJhqgrpkGCRxGBjkdcNmmaAoSivKZwGJFYmMOwtmYJzdjAEBwxTEDKNjXujLJuwtyXdSnVgTusiVOwvXYnhFBdRgugwdvwZvilUQvkZOZLCDgbpoLDhxvRZTlqLVntgbvmIaenyKFPYQSZsWDfkXliWUWoCQQlHNTPUCTHiExowdcRciiWBDwZaIOAWmBGiChlMnPoiqMHxSGHnxvyxshsHJKPIBQKUDaOxrToypFtIzRcIbHsLpRdmVdZxbGWHNdoZNekFHCLrhRLvROHnVwmaVbgLKwHCfkfVkGstpaFNOZJmbhOHSLyfutRsiTChRwJtSoYAHSgXCAFlaTOvSsxhswEScKeFnbduLgAfbLYOopyhzgpHxDWwxGbpkjUulKFRBcNWACBfOfodSDYmYYiTGdSUsSAsNnziSFKXCttpoCqDpXxyDuyYDQjcrQwULHpCyZvLUiaIZnmMLyJPcEVUxDSwIrKADqLPhGJDSOBygubFJPkyEJRXGrLiFKzwENVMgUYpQSGJcNjhJzPDWukNhHDKHZjEYQwwRfiMJwkjwkyQSBiPMgrAkRyBueCINFsQpiTVhURFMYsUQXMJmrnibDzqCaFeqFFUcpPjGjaufewMnlwYNFMnYIDzVDTknXfOJbUCUIBTKUmnLMsVFgzemMeIfCzevGAlnqHwYvNhckOscKOeLaMUOhLTwzWjaPBaxfAzHNTESZTtFSiGRSqppnpfuryYhyOSYbcsuMyvUqQCzofJDbubgbBsmXMOBGAZMlGtQmXdjCkyERynzAChshfxuwGMpxUnRieamgTHHWzjGhAiTKJcwsOYJTrLlyNepItDNtzLSrdnORQccvhIlnuwaEDWJDWhAeEGuDbTuuSmyvIrMQNAEhKaKyZxDYwzLvnYvpdshOCVbnokFbbxLWXFKAtlOfNbnrEJIKYtMIiqgNLzpYNtRaJuzIPNmlTqMLHpSQAqBgMNQRgucaOxwqaBPWAjkdwWbwMmAfdXQYZKrMJiGFpTGtTdMXoRXFTQBHVxvHxPAunWwtgtIOtylgiqEGizIYkIqTVhgDqJUVmbPWSikpuQgUBHuOZCNXPcvurLXhntauBsDrxkEbiScuUCcftUFjJcFxUaxytbYLadeiAoUzoSymKajohAastzMazDxeRKPzgdaZjyKNNeFfGZJizuMGrQVnUtxRMMDDUdljohkwyAWKcfespkeRZKxcdIitPbZHFFpaZfDTAzkndslGyZYQUcpDqMiqUTCbstLNRwzFmOwxgXLIBpiVrOdTZknLjAIlkFCchSbfTXvLIrbuQvKtnNJBJfoVnOtnObSJUkpupblnyCNnzfrwZYcfVYOPbwbPGsQtOEftDVqHpsOlplqUgqATdVNDeLBvplumkNHlsTuzeFJwVqcVAjKknSjgoGIStQxrWTGNGOvfkZljLQrhUxCvlGDgnlvymLpCaJBVcCvPLYIPCCegRmwrCYmFvgUezNFlIBjaJlglYszJLWDllxuNTDGRvcofaBlILyOJYzduxMzXskhFIRHVixfOlHiesIvMZMAgGxxWYBugAIiTkhuoHmkvZILhBngIFSEFNfpiIRPcpUzonAcUoOptVpOEkPeNcRJnamXbMsHAWHhzSJbjeWYJnyIQFzBqbBSfyXCfdvzAcTIWyElUjpATlBJSajcvEMIBMheDxkM</t>
   </si>
   <si>
     <t>2026-09-01</t>
   </si>
   <si>
-    <t>23:25:31</t>
-  </si>
-  <si>
-    <t>2026-09-01 23:25:37</t>
+    <t>23:42:24</t>
+  </si>
+  <si>
+    <t>2026-09-01 23:42:30</t>
   </si>
   <si>
     <t>{"key":"value6"}</t>
@@ -614,52 +596,49 @@
     <t>&lt;root&gt;&lt;key&gt;value6&lt;/key&gt;&lt;/root&gt;</t>
   </si>
   <si>
-    <t>9223372036854775800</t>
-  </si>
-  <si>
-    <t>rl</t>
-  </si>
-  <si>
-    <t>Zp</t>
-  </si>
-  <si>
-    <t>jH</t>
-  </si>
-  <si>
-    <t>Mw</t>
-  </si>
-  <si>
-    <t>gbDUSOtCovORjAECfZejWPtoElaaGmCqCTBeACAOCETBAtpFoqZFbhorSztueUznqbSdOxnHWaQoAEnNbqdytAxModqyWjbCyjxAZhENqCNSwuetTUuxxCHFCdZspPuGLFtaSagnzQvMbqQItOCEohVsIOOWEMSXYnDJsnDVAoukXDIGPwVzOlYqaSUeRHqAPYRQwDUNZtfKPvchLCsMHrmfWItGhaUx</t>
-  </si>
-  <si>
-    <t>FkolQEDfFTrPLonQsIyKRjqWawzihOYeDLgXSKzVskoxrthhUlufpwROczcDgCZHaRgpfKGAkihXLvvhOpAWakbAvIClrTYydaJjOeexbxsTSiZrGoHFwDpKoWhmqzqCBblnhrMzkYRxIauEuKlzhSznBsKcYdSTCYSRVaozVxaUtiOlyJCShEDjsOQCmZngMdSHcNHsiOAtNRLfienHRzcMDmOhphvZLPnMJXNNPEnGKnNLHUB</t>
-  </si>
-  <si>
-    <t>JKSLkAU</t>
-  </si>
-  <si>
-    <t>kGPDEbixQNBnv</t>
-  </si>
-  <si>
-    <t>GDALkQbGOtKqhHtHHmrTRtmbdWEiqYosWMCCGATohzKzzADWRQZdaaWWgldZmKAegfzhobujwavJChutzmRXVHTtAdxcgXGKACuPgdAqECdaatIPJtuFhBFSgIuKOPRukrvhKaBNPaCiWunAshEzARQIySZuCeIWYQaqbnLmOVYxNLBaRKGjmNVODRSpbyncXeTIijMsBPzRePOjHfiywjHFJwAqwIbYoOSQeWwaPjOnkoNgoTysuKqkcDdbcpaEYcBFqmoaoniSTsYhgeHeKjcAjYuJDbzmdAbyxgNBnwLjYSEwfJyLzfTVHnYgjgJNOMNAjmhmYKxhmewpmJwNzCoMwWZWXTHVLHVtoFzGBtpsMDVxzqlSdpLkkZEnuDbqOlEILfuStBMtkxVToFhzyaciVYTrzOZnDPCUNBAgAfmGShOBsgGzRbhqUkRGnfvzhILIXCVXInNmdJOVpRopHjtkLAUWvLQyMJwOJMGXLAqNYFerJtVtXzjMvJOSDrRFOSHTxnJoNlSEdqGFQETioiBmnVGMzNnzvZzxmQUgPdBciwfYazRxEPoOTddUqFuWtUTcYMvGTOajoIinlijCcLdHsYWRqxUJYlICyzqqVoqmGkTEybMyWtaZSgwcMZKsBlGrStmCdpVhXbKztVpFxGPaZotTlyIoTNMHoPjqrZIHgYPERlDaccclLOWfDGVxKiTztUBQstOBLsbBdADfMJnJOqifsicwNqqZvYpMZarOeZBXqJwUHsNvoxhXGsxRcZgHdQLxSYKujTVYUUnkpIWVlbYpMjLxgFshKPEsQHrXCODvdNaXXZmfxymrfWwNySULLyvMkAhCpPxfdKzKsJBfvdlENPevAJCDlxCqBvWnGXfDlLZrrtegyfamQGnszWWXIQjTrwwcqnEGQtbhCyiVPZjaWBxDyLfaNUoapqgSytJTOULUUrIPxsdAWNeIqrffxCaxWpVaDOUprvOWxzGcySlCGFSjSdrUsQeSLpLQsbkVwUsuXIPBPBnmqLoRpVtvawWazwWXDYRrzpuhaKaqWsGByBBmQFbpzVFDmYDFropwzWHbNqbAWrawpkyIIqsKvFBWoDiejcllMXZxBLREJcIUtgHDCskuvDvusBVLtQBLpETrZTXLXRXRTyyhBidbyQAudZJztNJPoWcqjFZacOyGUWXRtIXOcUnvQqSohtptpDYGkMTFwCkCuQbywdpVRXUkUsSetYjHfOFHWnjjvfVTSJdmfYgxxgzjIXoivTrLTGQaxdpRZfaPqBpboFuNAmYRGJqEPJAOxnOXgSPOXKqsIKQMwSnGvYbNLedEcNsGQepsRhOkrLjBPcjijXummHlMmzxBDIoGWqxajMNlKGkRXXoDJiScHqYpTqMRcnATyGgtVxXrDbbeKOmIsDsHWuljkhMTvBwiyVSAeVQAzZKCYtezndkrpXPYlLEbNYXMNMdtoSkmVFYcwWpgZxwfEUWOgwYwLdenmhqftkeqaVjiMIszajJzAwpTpKlHZxKNeYmPBmMPEQRmBgHEIPFbreHSVCVpsZmXrbAikjvzWFSXeqIcJJHDfhbSSZVJAZgnHWAgmnANHcTHDnMrfqWiejIWFPMhiXhUgCPjhrNDsyUDmCPetZryQEaJEzRhMFZvvHvXwWCiFPzrRJEPGAKYeoCfmdFoiveuxVINHTdBQUokfaaTNMBRgSdjzBbLdmmAgpmQgjkEKaNmvxAyWRIWOiKsdulAeIvFmCaDgHmBAwrYNCldnIUVMNhkXlLOdMWOcoxxZVTVcXaDBWhMwGOtNfhSPSYtywACFFQYWvqpmEDkNHsEnWBGMPsarnuPMXPCWytXUGjNVTIZOUjkuUGwbhNELJAKArPSKgkkGziXOEnBicCkrXgTrZGpWrjXlpRYmYgYUJgCdSWxUqiNkaMDWoBcYtMyGzsJUnIgWIwRYtguZLtHPxAHVPPRXRvUyXHZcNpRSBmClBEVtxCjcbVqbERWuobvvjxRJUdBgxXTqvrlxfRdRnZbNDHcSObHKrivYxcNQEleKdUqxUutyclaXskTNMHXkMQQYvTqsSwlUXhgdFVmfyOuxRgbufpPmfDIdphTrTWXKqdqzRSLSizysIxzujJmDNDDUbYoVRsmdWfpAlxeEumGaJnLTqUhZwNTTlapkSSMMOYiMBpCijvKdtklwfaoTQrDnYKCDrHnZYElVNeNqdmxJQgaIerbWEvKvFiwLEAxWMoCPiSjnyjPegPVdodaDwmyXJEgfYcidiLcokCqvBrAzDVHEqPELMoURFBqaNzrdBSibZHeLaVLOZQmuRpXPNGOOsDyIjzEMendBTIlchVtPAocBxqYjRijYYvuqjpQvXhSvqopUGeVZfBhteJgwiEnBLseUNajTlvITIBLwUmmfSQIaokvpWJWXWjGSetLxwdMUwQwKPhbmpRlAUQayNapftmmUyJPtaFRYQEDgeeUHizuCQxqMVwIDxpvtenlUTqZZdxOBrhXInuLANMtLjoyLFxdyUNLjrlVLKuDQYlLGRMfzOFtceVMcVabZbCVHfNlgaunedIaCqDOWiIURrXaeRwoIyDsSpLMVLRykJHqRKZxLjPETdjsruyyTEcyCQVuImmdbXpESYbkBjfaxokmrwoiNODfKqDYQZcQyRgDMnWOyrfRBjiImIeQnuyQVvGLroOtkjBZvVDIMYbxgAbAciydAEgQIeOIyOeNjqbhsFSHHuEDoegRRtUllbUiLLCGaPNImkOWGnWKAguPwltuKxDjdiUtpmYMEBYiQxkItbOcbMqNHIIFqSrCbevGndoBdVFdEtHNNbMpUKxxwitJNPLiFalVpjIjQSfyycwdClYXGSCSyHfRSffCSvCxAmTrLYVMwrEUOcbeVeNmBrUkIcKQDpvHyLWufiifiivdppYfYdgNcguSyMppsWhJpMtWliuLBooPWSMenVEjXxdfHCJdoKGjhgICQJXYFyuWUpiZtqGmQdHHeznQPTUNkzwopwTwRRZNQMfupbaLtCIJmkwYVrANUurVKIBDSVIeIXabWMljERcOSsUEwAunSUlnMdibOfQabXVbWMzoaRxnxYarEwrRodYTQMMOtZcYvJtJCqPDEvaOyamlgUkdmZoIFYDxZYbCIQjuvvvadmTPjToksaovKUCCGMGaDPGOUGRugtjNhVrHrqpbfebUMKDEArcWgMQsHNbnlHNJTBkdliFAmVQUxVyXtrnqCxPAyFeCpvHYpVcRrETOuvJRPYCXOqrhUdgjyPkZfxxczxgWLqcvIfyqvOlirzoHQKhYDGBmLTBzIOgRXivREKbMfzsQTVbNAbECGzLvhxeVfUhaQwxfKbqMmxBnPySFkbbZKXCseeRtiJQAbAMgcfcgtbDnKbxAgymdOXSTqOhWeQxbnIkKgSsVbMexZRCktCuFMyOWDpACrAJjkchdPEphIfxJnkEQdXkzBqULNxppVWCZAMDwSVDVfVWtEjjNAJOyyjKMijIFtUdDRFnvrMwoEbdKSWbuiIRUVXTxGyJcJXzsUTgWsJgtLBeazgYqGpxoUUXaygwunlkbfrDYoKxOGkIbgQnPrmzkmhRexuBJDPQUgXmnKMbLlpeDIjxBkBFKbgQVOeLsgjPeZoVkFWWrQdwShVgKZRPQTYYPwzOOpKCZSkSspRDWTWTzTdVYhmdrSzGxyXjTJlXFcMcTMKBPhWJoIWsziGXKIUlZYGmdLmmQgwyPTDVuWbkYJviluksQqKyYDpWYsmWWyMYUvRYwzsnNoxYZDJNfLUdvzWjXwdaKaOIgpHFEFjXVaammgifnvZSHmhpfflmrntXVHMYofVTPvpZklZMKFfXTMiGrmRGObftleccaNxCMZVxqjBxlLzWZRwslIchxZExzhWWqjJygJysYSnbKPENlYomtCDvjLzoRTwojVMrkolMsDkRerXPDiCVTVuhcxpLUUItINZONVNirfjWyWJRQesMWoBdhcEKjkCaZTKmnuFvWBUTyIFRjKzRbGQVwqNZrCTObNSgvJbqDIgqqFJrfTcpjQkAsZHYnUXzpHOxUyPeOOjoPsvolSQiSvapzqgPECZJtJGhjFHIKSHAaQDxeFWgvwByALUKNYmQMvetdTSbBYZgCqbPrgnKxQHZoXJLlZspoczfQrGytFCWxFzMegUzWkwRqBoaHfKtrFSjFmQRBSNclDExHzKSTjUpKshGVImWPfiUiYENzIvvSgpShIIcWtkAnQOBHdfhEAsnSEHPFxHrxcZjoejmKutLXPEctHBBQiQUYwdrSdAQeGHyjWxdbgDGFHnkXojJrPRAeRQXZzSFThUvKuCqyoAgrfvWtRPaIiSjQvoWPnyDbaOXrMIMYOESVBHcUTWbdqKwGouaTNLMNVjyPlnPUfECtdebkqDmLwlKvdDsSZAOyETDOZJZsQddYsaMDyEOLcKYOQYDpEECjaxkrBLhjsLRJbjfDhzNvFAPAhChHTAwJBljgfvuKzXqsCsMmcmrDQzPcwTfedyWPDujIYMmzqhgccZIUUJFdsWsVNmQVxOhqMgxCmvckeenQHlqYLbDqqQedtKGlhBAmKjrzTOKGPpYCREcTiRyazzQppddyAWOxCxChZmKlQthTnGQusRsuiVWQADMrvekYLgdGfFCrVgFuRkyhlelgwvnfVFAReukvUMlVEMGdzKCSqPPNmQmlGwzoJHXdChryrTPLfEKxohlhSGrvHlppROweaFfTXMRhRWZUpFVToiyrQgJyDbVbTQZVgfTKXHiBgpGzSWTHZTEeSBaXbTolVOjfkDmCEsIzhYhmSrEfJWcicTaVjcCBTUROwBsbLjENQvEMLuSWTUIyADWPecPGywHiHzzSaSwFuRrzeuvftMCsSNqHUcSGmLJnCRBCcEFCZHhMnCyywUSHdkbvymWIVTEdXhZtuOYXjJHZnAwMrFcDRyzkPAagbrrYZYfmpjTxMTcUDFRlIwkzIZzPxUOOumGOORWigdYrlSkHxAETPQoxjljSQTDKNsvSaGRHywRVWnTIrxabAEWDMpLLKKLJlCqiYvbFfBXusbfVdLfUGtivOpbjSZxfDqrrJKrZcCaESJbEaHcRCWsnjQtSuvKWAeTIwzcPPytMMBOTcbPdXysLDgRnHoOpWCMCMhjTKCeqoktdTcIHhqKtvslSNdYVkpZCldomXFynJNgruRtiQVDVzGNmqAdGjkRodcREkTLdzverqHIvsrLYdMVwWsGZPkUaZrDBnLBAOYOWJNYcZwgcszSzubDauNJsNchDXNhxkVWtVDZjwnbZTVGEovFEZuZItuqsotcgfwuKTTEFuWjtnWYaqbBwlJynnhmVNraXPMgikHbJzwWsGkSPXnnTGlovJbtNQMMgIcxMGNgTlQmxXnlTdNyftCDHBGPUYnEEIJkHnruIhzwOJVJklyTCCOzslGSnZWOfaGUNxbzfOGiZOdfICbKdQoedreBzWXCPzTIeQqpuUtKoyNQFDgzhtsIFOJUhodfxmnpYGegyVSeLMjQpTCRpkENPFtJyJVGItTtIhWKShPNtZTbwKvOJzLhMhRzzBKrmRNOocMWtbvuJZFPvrRyfoZjsGCeEhJxzLcbLKRmHuieXlcpROlajoZAVOuPttYIYSGjdrJeqUHVrcYKsumFeUNVjEForQKDUviiWSKnXuwrAiVXocOFCOwqOPThvwAadTfQdpNegRVxGWdVuxpKzSaYyrJuOoAMVWWNmEAmxuWdhKDrCsgRxyvjBNYOmFkmHDPxkRAmwzREdKTxkeQQuqydHnejasnIUwJZuLvHkrcCpDCQNxotGuvqRvgbSbEwljliYSYxtJPbqymoaRiayasQcSrrqXnUTKXAgRIngimfCbNDrUJzNwBKCDWgNGzzNSobmNEvdrbgPkDZzXMzNqoqzNLMUJjUmTLplQvRncWIFCkokBsWJJPmblrwypjlChgtzikhOTtHSTDuxnGtdQNFABvWwFbwKNWWXcQGmFEgjnzGnXnowltPFgdDClbntWkfLXlBaldvQHwiWSNzWIVbyELeXwuZBHcCgcGFczDYoPtxwSElhPJhGpODqWcjIUlOgpuGKvUzrplMayPpHfCLSZfUvQJRDgEkhozETpzqXWvvOrKMfEyOzBJFGEoAzhdtpCmhZPTiXWJaGFqzjQpgeVKXFqWJjfJyOgdDyXoPtnVVkLMmLdBSIAwhfuoMUrTTLHssQolPYVlqynJYjDBqpzcpsuZGCnwtsisKzktasAkYpMKEILwctGehirbSKINiEgAEVMzLDCKTUzmuKGcUhHsrLEAaRyxrwYHHDCccYmqbjSBKwOgJMlfOFRaoIeQwWBlsNMVFuIJAiYskzoJuqiMsSFprtvizwVlwwPlimzOIXFcqRDbSuPkFtQCKtgyotsXHTQWDrdTRZMdxdlwzEyRsRQplBakTpClYcreLxYoMpchsZMqIsXuYRIqooqcpPTPSVfoPVmAFMuddbemjCxoDVnLgUiMrevVJkWsdjngaDWcGVpzSOhKdXWlwemneMiIbtKzPUZDLynFqhZEbCtRqxNDJVwdkHtyjxJFxHjdETAFknytrMhbqopiABnUFJuuCqozHYzjdeljdIcxaRJKDAVQbwtQeyOBBUByFdeeWAfZWXIXIkHEmvokqdhjFEgEkTAhReGsLaERWQwzFSRUyWdqMTsavVwNCwtVshZUcahhWCxLhZDdbALDcFgAdSKlyvYOxbjotXNjsdeZoAfmKnLOnvvPOUOlOuFQDGmEciTNeEUJZZFjPSxRoxUlisWDeKJvDClsFyaSMweHWVBJIKQEPWRomIvqYyhlOvtyWWnhdIKZAdvJjAAFcLByRtiaxpNqjcQuiKXJuQSedgZYxVifVfMXCSENbuICWUJgJnNxwaYZIWaZeFBkxDhcfILWOAalNEIPSwvEXuNEHpaODmYYfZzIMuDnNQXiyUkgTOsBGJeYdtZstrhDgxxkGfrVSOEcUltANlsRpFjBZGbqFZKGoZFPTKZCPiVSznqSjXaQPFDeMxFyqcDmVqRssodbgmbdyixLWkTBqeUDjLxtVjxTUSvWGYuFzqdvjbWosTQZVLEGdcjnDpdgySLyrpuGrPTWYdFZOvDRzYhgGRAvkeRjEtGlNIcLTEpltBBOGRFvDeSfGQoUtrriFFvkhhZwCzwcvnTwWuYHtaCZrQkRbGQUfOrwxFOphFuvytESGoohfXhuWXmTTYGRurZveQBHXXUPdcvJcEkGTGnlElHQRQefodNiKEsvrJnNtarfhsmvIbUFoKxPUDvfjAUepqBMIOMRaSmwnjqEwrkkEuqcsqVOjwrRgnQeOHbDDsgDuJtGqeAYytxQKAgKoQFEfXlzrAKRZaEiNpPPQRyAqgIvDfQOIWiRMLgCqlcvEImMHqXPhVRlZTAswUcsgmCeDFcbrbrmEjpNOzOVaFBliYAbwBXvnrYxxpsLLrQVHheysQilnSTqvjapjLykwOsfQvnHuKEptgmIQWaVThuRxFUJWwzPHkZyutifhTedcZgTcoCIwEVeKKiVYElmlwqaOFPerpOOBkflgCmDHamfFMIRHcNpSDfPapnyrwlNvMYmHOQIEXKcILzNShvBxufzVNyuXCgQHocOfwozlnyrlsYKaDDQoWTBhUGmjtgonqZJkRMuYeMxHjQLzgEaULeJYvyWyFGjFbfTWDDrxryuXPkVbFpMVzudqzIdOHogIlYfPprunKQdpbhJaNDJrzrNlXtaqmvoRPUgDhpKZnBVObuNvKCkEqLCgRsZwZsrhWYoDTbAYVQSOzIlIPCrFqELyuxIFKiFpcAcdDeYIdMCdCBzVmUktYcqrhIjUqaNKjdOEhnghaiarXiExTHgLnDcubwcByyumjFdgSmAVkzsUyIixdeQSzedvXMGmNyXElBhSbEZrlpPgcovNqNctkhrxApdHdxLPFvpCjodYvCaeRVYQJhwzQunzamTYjgIeSzpkjmDPgnERfZesvLWuajBGPXKlTqpARweOTmjDvjCfOFRvxNwbjGFQrMVuWLaOBZRVIWfpAVtxkQnAmDuqdLXTXbCemViGDaTaACIePTONXFyjYeuiKfznbyMcjIYEFWPnvXKdSSdMoRkbNotmNUJEPdkwKDvgFbPUahMMUtvCWZkEMTvcbPAheDEEFepLyMWIPYpPIUjVctgVacEwhnlnTqVOEHDEauvJoXfxYkNsbtqIEmMahjLVsboWMlBCFcRoJgNfhxLEIfrHXbgrgzGlTqYmjXSnzwAUKUFZyumOmcLKgJdObpBVRsdpqlnqipoQGLdZiYPobCLhlCtfgsJulSmruSBWaEhoEgmuVQQbcsEIehLtrvSlcklDMIKhKwhcHkassdAKvcWUScEtCzEdRzWdJodEJnoeDYoDcrYMFuyCOSILYtNxwIkCutniiEoJtTOdtvkeWQAqIOorvXIWCHYdtwMwTWNwzixjaCZOPeNzXcSHVVqeFmxjeRVfJheZDXNVHWIYWMEkHNdOXgFBYbUxypIEMQnWUYCDykZPgMrAqhbarHsfsqYUyVSfvOBBayapafpVPjJmyjKyPbseHxwAHMmBpKfomjZJiotDZLGMHqwbZPkNAQNZTuSBhCMwHRiPvXXqtRcZINxAsNqHTUrJjRraeUepeBSZNGBBViqYhIyTZdKdGTQiVmbVJigbsvlShXuPmchbBUIGzSASVCWyYjcYeozrXSUpPugQKsewIqlzLfqYUOQsFLPdvLUhGpzqWKNoBGrDBBmhNStDFwhWIpNfUgjNEAwRbEsDAAFBSTTYjYqPqrsRkYwTUWorJwVQggquOwXnbaiNMUyvsTfRVQZfEQARFKoeIinmoHWdifVCRUfZifXUJPXOGcbLTyWKDbXCRnQTxulLzBmUIyzlHijVSXzZsiqGFyLXRlOdBgoGqpxHGbyIrGqeiKdAsYXqpRVLHHrStEueWJpPVmAmagxjGERBQEpNzpyAYAZPMBbdGCbEVojcNnuSkxyvXJGplsytvJdodguKgzQPXJPLwQoQvQFzwyhKEiWVrbBSUVgJUKXCstbWMnCzOhgHeVqqNPCWtzcNkIHEGUwmjCeTIkAUdLZCUJyQtKRQRhvZIcHVtHtvvcYvEFfVYGcWZTRkCGlKMOQsoFgdjJVYRzMqNWbahVysSkAYYkJtxJoRuEoscJrrqhuqpFpROZxmqwlphILlsIYzaaeLQroPiqqwTHwzegtgrCdNNfbGLAEYGNIYxdEyacUbTfJHNtkJwHyzOGVIiqaPiJrkXomHrgMitSvUTOLpLKWWADODrqCouiEdBlFPYQJDDTxngTimiIjcxJMEOnvNGPvUTuVExJJagucuBbrKltFtnILoJCPzkaInyjHmIJbVAYJjQTzNnvhCuYPNNlyZoHOfWSmIuyXzNUrJtgjLXOvHszjyKRdxtUkTSqHtPaWPUnbZGrbZKwMumRKDRdphKyOFOEhSKdSmgeyRdTddcrgvIexGHaVtXQlHvNJcUoATnRGkxdxaHYdlLQppGQfSeYneqxQMaJVsMXpPeGXHTttVgBiRmqGEAMgLHhubZFcYgEnqAdsXWkrcVZQYkWEfFojaxECklqzDvCLyrwwBAQqmDWrWPLTTJZhjVuWUdYPWPdGahMoXEpuZbFQfzZXRoEbcVvLwbyTVlmHsKTtyDIZxcXUgncOwIkKiozhsZnzWVKOTnOGmllspXuBHKtkymWclxDkRUtxHDhQBjpMYxtyJfUxJvSKxsHjwPGMPmVccPplFduJDxYJyKmLKJLTVQtDzNaoIFrajhytiIYLqDPpeJMpuDkqEYaykyTvOpztklVaaLFkxxySxWWQlsMFHjOVwhDmfmZVrcpPtMuoolhnphxzWXezQWOUBhtOhGFCeUgjoFNHLjCDjytvaADbPDDKhGlwlrQYqAmmOmfrqMJSflyEFvsLeMNsGPpCpJfWkzCjBTTsKxXtQblXPFHMuPwHEJtAAbDtpdCHuGtTXSufSJhSTiiWzexHspHMqFTHSagQAZJGMrVtDoerOcnZnyRrdgGRCnihgVDOXdvXXNLaJadnvECsEUQPLYCWkBEvwckwpnhmPUvpkWMKvcwsaZXlbZPbRxoOSavIuAJNglCmYqRdFuiWQPbFzCSsBABcjZIhQmDuKhdiWjgFYTiSZqpwnklqYrejNaOucRDWViaWQDhmRAhdIxEaMgEoYGMdTVBYsAesuqntEtFsuiNVzqONwTFRtjaRztdOsChbzdXdkvDIEFVgaUJuFSKdHxyGYLWHjoYMMtVPRHbMCbZZnoTHcpFNOLEzeQQDwSuAwJIMZHeNgibveKNNMJlgpfBJnPwueGjxcikQiPEQdzepTTyHfCCQtEBvrkesEvQpNAWLFnYrdQnIyGHUYQCuQZgWMsAsbAlGAJgLWLedzCQulNWJRgzFgUJrlrBAdShuTxYyzOkvNkskCgHGVzwwusMOqHyZjHFVFbkeUNCiXczlzQUPXsGCzExsgvtJPFVfcBLbseietZpJfaAENAJoiceBchGBGaTbKsEVWmPMwLOehzkMRNRLiThkHTrVEslAsQlQkGPuFnnjGgeOzCqAsCKrPIzxvOSkytihcWnoogDdAwhJTVwnfEfLUAHYNsFIddlZhMGePcHbaiNkuRcSeHzkHuCAsyMOVitokaBvyLxdeFFwgEiWBdOEyGHQcSGAKxHhvxvlUObzefTFrREzqQfpHQqbXZhzpTCjIsnqjrAPgvXYJAAuDEavxiaePGPSXRLCrWutqZkxxBWiHZWhlbWuCyscmHKpktyEbumugHfEfkjZUYzSwjaGMygcisMbeIDceEKeUTIHPaodhtlRdFEkBYngcIFGQGqzzGloxpCtndlWbrAPUSESIDecdmXzyofsaOwDZVTnQOKZTtUpBTVubVZCQhybPijhSAqMOAeGkWUCjdnQKwTiDtQCRTSzrpaVXUOluQjyZIPxleaSeNfxoKwOkemzTuJWqryWXPNTOCWPNubkGPjixUDsgWGMbOnTIKsSXsctKapNLaPIDOsmqwuvkHRIlXSjZnVlRTkTQMjFBDettIiLxEkTOSAkNDcfvrUPmAarQPBHZoZbXfTrUzbymZCqOJeFvAiqPrfhYBOefecFuFaDaYtHpmKyooyOgDJNOQQKgIqIcMFLpARVzpVniyBKXaQZXMhNvTvKQMiwJgwYhAfXWMPBGBqKxWVWvGOBmhSriUMpaqoHvJwzEcffWiFzgttzjaoDcsFEzRUMeeVxKqavDhqUeKiWZFuGwELEhSZCmEWgBbSosaUMtPQyLOTOiKogZUTQdicbgnGanfTkMInQJgLfegpVRLBPuHgydfVeIbZPeIsihGSAflcUhVFmkztByjwECRdsccznrrepHHYHrURvTgnJzXyTtEcnawsTHcksKclocYSPBqYSPFAPGgkWzksWIHliSHrDWrmzfqzYEQhaNyqmjzsoXiQBJzAoXrogbsAQOUHLWCYoxOgoRjppHumBJZaxfyFlLGsKKvpOEAaKjmJxjfindQBNZRTMQBRUCVZuTydzOtdZeffxkBddERUCidzYIlnGlghadvyskHfUZtHFCXQeSpDRcQXXpPwgDviSsFPLFVsBxMvMloNzsvnnoKREPydljAPSAfqAVOkLCfPKyDnNlMPXfdSfZplqHmgaCRVdyfVyOEjaNoWeQQEQAFOtmsQqGorbKKXdwOkqmColELKeftMNrZLCmfubdsFzSwOiEfSQhLkOrbrPEwDXSWdylZyfDqODmBNOlGhJELFdzypINgvQQJdkootcTxNdxQwNHujBRUbMKAuKykjjSHzXiwYYmIFcfFTVdnZkjeTdZmwhWqLeWxuqhHVCfPkperVnjPEgCAtqVeADcUgINipXNPjmENbKdzXlPOTKDvnRBghgLKGhCKNGjcHzCMjeJgLQrdqqMOkisYydlvFBCNbVBxQWogASqqDzKSbejLfDlHZWvqCRmmtITDjwCjupsDhTJGznykgvShXQFuJXzSfFgvjYEvjGxHAuScEVuJyfwzmDqAfQHzMBvskjzpnJAMIexrWfBDLTUquVyneohUGTMGyWzpQIQwCFigApMvCnqPilgTrEJhVguzWkTzZtStdyLOLwkJRaIEXsnVmnLEoqLfyaSDLkcNiUavKFiGGZMVmKuwCxXsILgkETGwCyHVnFwycXJQpFMDEclOCSIqgmPqRelqqqPXxruvqYftJTVWcoOniUZnduCSbDBsVaQXfaVtowWTSkCLiWrfCWLYgHyOQRPOgdKJeKykCsspBmTkdLVNabDnSKibYnNfnjLSylFykgKebVJozJJVHsutGozdmMPdAqRtKfCGiwsYJQGpIOFBnFKDQnIgZAvCXAaqFcpzdhiWEXMPvqUkAHTnEduCptHjUfpUGLJwxSukucxcADDLHWNhqCpXuxkakpJZTPJuCPVsPxEjwozzGdqzQWOUfoUBSiLNCktJkfkmsgDwniCLrjihSQWvYjzmYfSEfkyrGpwbhqbueqrkjIikhmqczlHpmqbJCtHtJylKYzdFthwHKJqiceIiyVulEJvJGoNwQEIvCOkyejcALykablBGkmfDekFFVLAjNgUCiTfkhqwSxTjmblkpdXONszyYObErGEhPUpfxZTbXKXdEvhuJZlWFKPXdCHfQhESKhnYFnELrHdlnpKnsXNKkGhfljSkyqnFJLiQEfNOQicDpYZnqHjElbIRPcwqBnGjWoRzDRMWnPDNwHndAWuqnhWFYQTkhQrkHYTkNaYbQUjoJUdBvhpGwTicAeYlljJcMHFdULKUyQNUQctXujNiriVmaFmfJFavoLIQlIXFzDLvgNvEIujGjhzwAsDrpeKbZIKDNNMLHNTThPSgcLrCScLGvmCwGejRFQKZRhOiraJWFObJrrvoWKoImcXzlmFVgpAVgnRLIFNVIIsuYfCLuEUifJPMbSiepIpwziuZcQWTHCBbWzOxHvUmRKHatwYQTLHilivPRlTFxItnEZQRlTnfvpYmGhIQQWCtGQBdDSOUrnqGNMCRaFPWEUPTSbjyyRQtSxFdCypqlCysEUJZYQRLSXpZZkJRomZssOzOkZmklnnVczEXOlUskeQzKKALfmLpKdNcgeUnHqzpJxHzsKtLGssVDzfmXIOnjFIweDRrAubXRUmsZJyaIukeXWjIULNfUtsOgjRFQADvAzypwQvGBdlsGRzVDYhYFjyMQLkAxWoJgjHgOXrKoUjrPmaAIPJaVcvkhSoElfkMdNRRUEfyWOVmfvhrwpGsvjsSFirZbrSDqvOWMFkRANedupDDzJSepOIjUzYKNiUBcOREiyrDYcfFyMGJLdBuAMxunxZVDLIbCtxIutmqBreDCtcUyqzrNevyaBGWExtDEsblJSsCnjrhFwxjwKMNZQFTHnlXSjOsjYofgmefeTRjTHlRZVnRhHPZXHDkChGDjfxVInNRiFFAUkeMEabQzYGJislErueOiBSbWiWnbjUiXVMRFhurzojeRPIoxuEHYGtoldovcpktBhuAWujQAIdDCgJrmLcvRVdysKnwsxZRSczassGJmJeYmUsIMloSeIqdemsvezJmJdwXrvrXJBnDIQtjaupQSdxcRNfLFbolHkLTLbacqhIULqRzituImAuBQckxImwxpFeFHVOOiihRTqXljiMbBMxXDMwkUhcWDkPykBxMDnHiLKDKlFVJwXCUowvUTYUiFFkSgjLEEImmxPKYJrTYYvVCRaryYxtuoNccZRYsTqjSzbMLBtdCyljSotFWZQUJcQsTzgFhscustgrAyLmYdFZFEdSMrCzemEfiycuVaZPeHmulalNKBdEpzAWPJDxjAolVXWXjRsYGIVXAlyEEwfLnSxWztjeoJnrnnUTpytnqVmZzsQkUyQUEslgAZiLikXwIArZoXQqkQdrQcVcwPdSbyAlxuiGqvuCMEkGWdUBxQbGeTKrnefcZrAblTgsRaOpZARSdmYuZUKvEaziKIQvCrYxwHaQCLXsDYvsdftnFaJNaWMwFzviGeVfbpApKfBtusfrwdyxAQOhhyNfeFNYPYdEDSLpqgiMAyffVHxkhaKoNwveUGwWYDaAFnozDeGuJpxdVCDFgHBHiDfeNTrOLuyaBaJMtbNIFzlrXlaXxEJOubItHsCllIcJNRCYjfepHWthWkQsEnidlatkyxwErdeVyxkzxrKleZiufBsLlSofsuWtOUiNsopohaErYpKvVmuzIlUBzoERGdYYZmrNZDFHVpIxcmGDPPcvdFZJyvMyBdZNqGjsbwOqawAphOxjMcsSxoBQfTgBoORmAVvQsxQkAXgilKkyxalKicRWTerKQMfITgWAMBQLyeXjnKUihyIWjoZLOkUtndziBaadWMYkuyCPQJSuLqajTIbhSnrrqMgHuDmEOluXCwtgftbsnrnQfrBwweyOsEiGoNOgBPZkkgyzbUjYOslmKCiqAUzDyzIJNTFjbcPEHVQOAFjSjSaBdjEuMCzLqzroimGemLyMsoQriDaGPLwagcQHOtMrzIlFyxzwEYGLTZHdlWvdEvoYoVfuFeluolZozEONAsRCcKKsqCRApANGXNmuLpqrMZCPSBhoxJlzayMZFuTLHcwwAhJWzKxZenhWrsbBFieHxxTjlJskhsmDunitWcgIfCdDlyyNBipdxhewUJqnPcUqORqtsNgZmkxjPqpPsRiETFSvpZCuwAJXkeHLKglbKfgkwGrKXgYwXOOndyvXFrMASzxiSbGMQkvGoReSudNNWiXWzjelqUwpCsZpKesDeYbkRinyJTbXFCJxctnucDpmLNMWSIbJqzbsSVeIeumXxiIabzQPKARCHYEPTtWHYUCkERSmkRDbpuhaJhWUmFXrKvXZmhtHRLxrlTCRQRyBLYRActgGAiFKeBVDNjoQGkYkMWctmhYnUKLVyWdlZQomPcwLgHbDvTQuJubVcBYArHrWhSvfGGBAEeYEBFlqloAuUPJFnxtIYtJkKhDhBjjIeuOnWAEcPpKhkkkhBBBodmHqQXISyrvvLzqnBkNimrDvbMPzfuxEtIJvzpBgmsOXLhJbwljetOWaVmLuutNweUBgXyAteHgjNXWTbqwymWBDFeYPbTwtAgVflLbFnhsdQUIXhzkFiIDzHlJLLpIryUtIxaDGWDfecboisHDkQpqeeDiOQBayhCdOpgibKRqvHlEmkRVTSYRbLkgZIAjvWkiBoQizHDPXQUyfuKqTMQNBgglAHUcOzNGiTweCWHFNrQcLQtuUVwIaSwxhRqcdHHhqMGAhyHCBNjDDGwWnNIuPgaKqnoATUlHBAocRanUcuTLiQLsuELseRbhtUMqkOFkQFOoAyRkskxmTdTNrXQnWApljsuESFrWAkiQeFkNjGLBfuqMTiqAKRrdxowQnhKRkbCoVzwZbprfOZllUuMfPuRpAoVbyaOTsLJdJTdcvDQfYMhUfGyDgCqTzzuGDnrvYviOOzteNVZbmVzTLOLltNsZQENAQmpKgAFuTyUXXWgjcihmbQnuxeTVaFzSNXyWYVpLbNhmgqSQWaNEOjzMFTAMHaxbYcDUfdzjaVOqsiSQFlmbBYPxhTdJFpHWwVWQFnZwYgpikijmjWHeBiJQsRzBgdoiEumypnphYlnpTXiIMLfRThezkCjwnCJZcFEXajuDhSRWxCktHyLaApfnBnBuGewFFvzzHrxMbwmMvjZxbTynDWDccSVEGepdNPskUKMMrymZHfICCNsKZkaLPHFjOsHMpQYbvPPUzAkAsSQEQhzJxrqXnZncHAPEtgogVEXdKwpdscWLdWqBzHMkRJSsZzuArHuxduwaouwQcgMLggLIskdrtLfZOaOhYEJqYgFKbKkzfUtpGqVPBuoQUyPAMgwCkUVGCxtZhHTuZsnWaXwxxctJgjoyzSmSzCEhMFoKBcBqFsUZvMkHpvNfzdcnJrqVHuKveOyBNVmMoDzEFljgpwgUxgptTRtTwOWXVUGynywrHpKZjHiwNqFfGnskESjHAaDgTNRlkcjocIqnnCTCPlXbEXDlYEajuxuuHRFYqNrQWHZhtvHcnogUIvCRhwqswnYKPgLXKDhLJqVWUivoseNQPciQaVYeqtFeQneBxkcKgVICEXlrShYIqdZhsyrNMaDlVrfQDWsYlAXNJtuqiYZkKJdPdlEMZeriVWuLieDoqjCWcBwPjQiZpGVZQLMJHnHeAwhnqwCBYyAYsXCorFzslQGnjLXchbcRQGybVewiRJDloAEqfmYEKVpjBWTvOtUPfiJafvQwSCYAtgtCdwocCmgOZJlmCyCVfeYifoFcmGVJTuHSknwDcXdGgQYnrrCAbUFHfkCwoAGHDBUbtAZmAidvOlycZffjJiwCstyjDKcRkmooCGGTVoSCfYmIQBgBNuHTbcexYytbSjbbQIcgSKgoLPlNAHgoRmKqVULBzAiCxEbryMustidBkSVZPbNLEtLnHzEpWMYETqsGfgXsEpYdQkGEOGVashaRhrQSccqyIkRmOgMgVxfGkOWkekQbssNURfPtNQmJQFuJrCwswHEHcAQiDLiKpGibyPhakbULIfkTsiUVXRdAPddqkQWLgFDRCcxnkpdRDYXQetPcEkiAACEnlaTmcZaTEFzTqknecuSfxoJcTfkaVdGRcNbyfaYGUxLAlEGQThZXaqbspOjfwNeBURBPKvWTaBylnUKOsskwqDSXuXTNCrLQToPyXzrbpbQnwIyGDoTXsEgdMtwtjYqMKDfTacAqmWbpDyWqnrWJJMwzMunlsZINgdwgCiSStePhTmXvDIJaHWhiPQmUNflsRkrwEZLRvLhRzbLQXVEPPGnStXTPIpjAWMAsLOABjlOvPMlQsQIwVZeBUeyGRfKMJxEBgPqXwArVsaIAdFVOcPERcyqZVjhjXtZuQqjAeHhRoBYIXJOwimEypfgVVCyieRNCRvqzxQifBHXvewVsAponFwdZIrphHtmGNGvqHxqRXJNeRQCbDoahcENotlBwzHRaIlgVmAZMncFbOiKRXadXtUpEtQjGHJBpyMgaGFHsfCiALtiolHlCPPtaJIrHGUltRTsXyEhVdTwTULcBXPXjRkcsApYoBmcKrwagihnUOUoLBtAejAzUmfjnIcIooRXpuRZrASjstnXyHyRXKXIVklLhkmznnaCdshdjBGatrIkknKvrQrbTwbSefrqrNGfVYHmeRbHDNAcKzbbloqSayIRhrPPliNMUkcZcKmwbSJIEhgthlTYLuRxqLJzgTOYZxKfqrSLpcdRgFpgZEvArRkRQVaTcnZJsDlTQNcJlMqClxoaJXUxEMdVpEMsuUACWVgeGxVJrdNfUuNexoGqypRjYSYMBpUnwXNFEwmODncyCjtGsFNxKjXVyApROwsEklcpDfLkrTrmIuZUlFMPQpBCkovaHnSzOttWboAItzPGnpMwPCezkOIzRjoWlEWnBbXUYkXIyoRcbTKaYvgAJOjpHTCCPnxluAkDCjvZlfZcQuMRZeJIulnVwHwsQBJqnYGDHlnwLeCrSoWMosKwUoPqARXFEuCFGZjcbWxUYZGiTYUvhvEeQjQBUNpjciaqUiCHCiaXIHjLGkNFJCAtCLJwzjapvTFBwTINEVPbhPLEIbFWyUlqLJKJbzFXPXMJyXugmygBSwCehrhHHkiTSdcOcYeNdDHrdWnTPqkCyYIjOSszKKndbfukVShKClGAlZeXRKKCHeRabicHeZJGURWBVAVvGIYLlVhDEFfPhwOUYWUXvERnkXmlPcZHatZZDzJZINzHuSroTtZtZbkBIMCSEiNoUpZzFtwevBZxvCySwMZJIXQQWimHyqzuyHfOdhumRBJdRisMhYAyKsWWasSGksdiQgDHRIIyeCzzmZMQlJkJfnQcZbfiOmsMVGsCsVKWZJWvaDOPVVMkfDIwJmnWShudNjoyvkfEStShfUIzuBiEruPVJcNQGHWVHymuGXEdSiqIaHRaPxJbaVWQJwhBYlnyToXNRkvWJvrEfNqexbEgXRDcZZGKTMoputaWrYiIOqFwRGoDhOlFrchAAJgbnTgFsoNxlkjEPIHpacWaVbJqbSoEvpTsCFVyAehlBmIghVyqAtxhxaUCizPRbFJMHLNXmKCXhqPRFEoFWhqflKanzBlfXosdtFRXrBklyHgssOQSZpMVNkYpunWcWCzIfUmNszOKeYYbklUwtDatJnPxOpJskQqPvLERmQEoQtbQkEtbCNmLsJDWCXDvZEbiapDQApuSxSsNbYJxVuNvoLlwlHgGIxYdnhiGMdRoBoDJvJyEfMecdqitMVDpEghReVThxTMhXUIgyeRETwpBIThtvjnPJpPIBZfDXIWpcuCPBxZmqZTNTlhThcUJRZMRmTvJSuTVMLNDSvoqvKOBPGKIuzthpEGboDSOJaIbKEDkLBersoIbbznlvOJzyTnHUZZpmxJJKxVZEQaTVlaZujXwYRFiffozHcHobsAUwsZZElFilVMdRSmbZAeyBEVvSCcITnYMedBPCXPYQpOeKTUFlqlBqNwvAbDCHULUPAkossAOzHiVvXLnaKtiPnDmUkgMKkdBuejBVHXAETxQuyNyiHzvPZXiMzcEhZGTuDzIagMRhSEotJahNKesZIgOhLwzRMWWPwHgyjcdtphlGBoWdOGupqooMjPrlCtWhmcgauNBuTWsfOtOnYAccVlhNYyBXlTjJrhxyERfmKIHAEqNuNAXyCULsYeeEfkhlYnJiwGDaoLkvaAqYNpYMrkIiYTLjcqTDhivWgfTRgYdLvHwnPVfbyIYgEpTLZwChYscvoebPNAYsFxpvUwtCKacmfnymgBVcjXaDdONbuSMlGBJxenBzSLUsYyfIMjpwMWbEsJCMMAZNkagdckXLVHDqCJDNrFstBKXCcdHGBavpuzsZVEFcULAdhIBmWpYVkBGkJbeBLHngKqSErxIGQJceveIMxWkBJBmPyujCQMlIvHhQTyRuHJLPNKdAUXnFUDSVBcvRMPtPyEeTGaivRWQfIOnmoQcMxTwOJWzWNYkMpYwuivXvaPvaLUacWCmDyIwCnPWuEHGKnVClISOkBOrAAxrJiColyLABnHWequBmVWApGIiJbbYlFJjrDaEfrjdkQSXVGGtYXzxYvGJFlxtSdhWOnihaXeQxxvBSZpEelMpxaDmuVNJHZFJDXofxgzTAoyDMZtFyFXLmtPmsaBJGdADWaDYExnbSiANidXauYJpUXplxrUhRaAQecHAzDeCFimIazUbeCcwCDCobcdFwKMNfTElwUnLOFroXVihVdSMoYdLBQjpobbXcZfaekTLdPulJQzHdlgYYuHEEdKZTGmXWhZDafioJkVASvvJvqqLOIUCGtXyyORDiravlTuhlwZeGiQYgnAUNbakrVZMMSFxFJkyknXwQCRKsyaVcHzfVgmoSLyUEhxNcJUBpTKAusUIYmimHkAlFCTbXbzBtaVHyFVOROWfEGtvyrGvQCDHUucpgtTBuazqBInKgrwUCoWvUTtEblGGJtKSyCaGmAjJsMGSIGGrWrmAWwQHMnWThlImXnZkdsYGEMTnnhlpORScszpLSpFJlIbDxPKdeBJiZVXjcyoorygZNgakRwWqQGDoCRyyBAickVtHXyVmxoINAKdsITHjoYnZylRQURxEcWYAhrNBIWedISceVisNcWJWPYcLLdTyrYmePMjEvrEzozCSOPUSMBsahlxoffUPqRvuSqBJGOBRGgdoEOicMWvuJnFKdFjiILNGTBAYGcaWRBlOZFGeduIFLTVjZlPLqcIXSgjmEDZdAryrmNrPUwPQpAJpAQnbWTCewAjgQXbqGdPKuvYLsmzvptZSlayfeAECTptEtGTofciKZXtkorjglKxZgjRTGAXKjfueRBauoHSprPUIgixRqWUGtuDTpodjYoXJTVJjguVstGcAWShKlweMqYZeQZcmHBYUzrkXoAOQRsGgYIehQwpoovucSsaWZjZNKSPNswAlprRIadyxMFUzRLUUEwEDcKOBWIYJWYtKMuhQMckGhBIhULxXUtANMTAjnbBOAghfbQcSPMXTSsRHmsfesiZrxlHwLhWVOLRktEjsRkxxbpRFenuBlfYweCzIUAOrsNteRDFSfdEXQPJHUSHjIiAbiFILVxxBKHAHfACNoKuWkfTDnJEhJrmcdAkfDVbAJiqFdPyXSnrnmdsYXqZpVzoUYMifNwMJpvWYjqokqgosIelHqMPNjBFTXsAWaREdoGRDrtlxmsLlircykiVldIRvVcfjArJsJlzvypwczOKMDvcXwqWDasOjbgeozuGupKUBRTDAblqLhjwRrjZkarXgWDFaGeCychSwueJRGCQRwCESJhfwZrpHilyEirVfUOBykIIHwnSOYnwXdPCDOsAsxMptCVPXYVZHLDzDGMFuAJbmthxHNOJqfFZVoQuBcJExGTmmsqkeglTKSHUygazaCeZldOaAEVVHthdKgfCQdWRhUvhLJMKqYfUlmFLudQZstfRBZCaRbaONTYqvTCcFgMVCvqaQXdETmXBvTkxsertGTQYlDKIOWNPzOCSuynbcYfYjvxJhPpyTmKbFpDmGkYLgFlsYirAlpTiBOFGayhpxcErRSjYbPyeSmihJWtudGCoDMFHKseHglpZbyHjgLFibvGZmOqXaxsiaiRlBtvmuxMjeOFcVbudvDRiwmgVFXuNznGWWsxGsiYBpXrfrDDLkgJMRuOCJsjaXedoDHWNfixMQRLmqleUsinurprhGDHXVRkGfFwAGpiNIPkJrqfLvbDUYYbtPtDNzJdzglAVnTxDyWoOfqbkCmWYJKPudQrWSxOMyNDZZbzvYhLEnnoDqyXJVscevFwnEeQZLUmZMKPREPjmqADpiwZkPYkfXaOlvtEkbvulnSgGjQlQlElbjugUobPvGuyXzAIBqQgBRIgkSTErQoHnnREvvjNNUIiIhAISxhAEQvtCkNyGIrAtESmkHHbhBqduXyskvAYmtvTlQmqezOfNMSYDNpfYzlRGsVEwpWwHkCwlttLPZsvnhYritSgAvWquTwQGeTwRWksxbYlnwsVFzCOpldEiYCtIdzTwWvGzOCStMUsjxdxYYOCXmZaiQFzRLjUmneXAhzinyMGozNoWYNDPoTBnHpEjZcpcDIGVjuUwSFNJgMzMgmAhMfiTMTSHLsdImFeODzMSATsysInbQYpKEOhAqUawgmOGBHjnjnQYbEuzoMfHTPPUeIiBOxvIbEsrRloBtAwOtRDFOQvADPQhBBZFxDteZMrGwYtnPPiUEokPnSDFlwjYXUDSPWnrOtmXDfVjAiIBUIGKsRuOQQYOWTQQciWqdikzboEquSSEaiwEWVRAppfiaJVSzKnJoSWBdWoFXBIZxEdvOhvWSryAgbJaoJzxgwlSbmTLNadEqKJfLboSKAvnQDndtZnYraIHBjXeoeKVaUiRUoROdSuCPUSUwCAutsRjPiPuLHbDndiOmsyNcZozPOwCiRsgIPRJnLRgiBLhtzFOEomXHoaBDUDXmKqGKbwXaToGlPrRSqJXzlooyqULvmotrbsXyGdKmKIjAXCbAaKjyPaYRsZpWPQbNKgcxmbFnnSPnwcWGoQRzbACTOJyvAUnBnpgqHhRBPoyRWxHdcMxUyrBacPAiyMIZFDJggvAOUTlEjRxKiqAWJCKZciGBAUEDkBoAZoXEubWHRdUMhhugUMIZQKIwQRBtxqlNWYJtAdQEWfpRlUguuqUPBnNzbzNbjvhHhviyZctWfmtkWHOfjlLVckVfsnoxqqusNuKEsnkNjMOfnmCVsRxpPZpDKFxstxavJsSICSLCEOrBgKXArcZoJHBFRGJITwjiDSTDiRVFXuGTwHnwPLPrODGcUUOBfkfzwWJvXzdgvYcBvimGjsSPlmwPwpvdohZajFDzPMorfAmlyAHGIOeeETuAqbvNAECrtuRGlIfVyykJqZOsqwmFnFmJCGJIYGnJnoBZQORtyMoNoCoJBvRjSWZZJATFgaYgCkTSMAfkVajIcVxBDdvjnBzHmwXSROmvOPCuujHXMLEkKeFugoeGLGAWmuBKLpGRmTNSJUIjCVGVyBsosrnMalxhyJKRxNozKXPGqsXKjbTLwkCqFQXnthfygassvmpXDdYpXfyTvnYbHUlqkGyhKFnWLVDbDLGTLFihTCZeHYgKvbtkkNilmFBhLwcVKdOfpjjaoJjclhNrNxnJuTfIGuSKHNnDAEbeEXxmgDYHaLrlQEVjYwratGhNqDEMlUSpzrcnyPHCWEkEriTSsdNQQDySpDcaZSSPExHMrLgxPLiaqDdZxQtfEpwMroOinEMADoLolvkkGPeYIDVPAfjGmoZRmIdooyCUkzqSxrBeicweCelmMvfYJfuiIhcyNyYGzWBHDihSnrKqUrPesswgqVyrQPgwhmhvyASaqRPzxCWFWqoKplIIvYokExSfWZNsCjKwxePDqOqkQnwSCnQxnIuhYPqrsSzYapyHqZRHWRRVFJfWtRMdUShORKyyOyplYazNewEfNtaVLAkVekYBfEMPvHbqQfIoaPJhoDFUBPFEgTxpmnUMZyBwhjOBZDLlMrVblLGvqLgGtZKWqfqoqGHUXaYUlstbPAnewiwYXRIwCHPmUUENCzfgOMuKPkgRnpNmxcWcNhGUhVYFzKlaBdjyfOZFXHqcLsQpRLLFmkeQCPrAqrRjCAguDQdNhrzgHkfputgmSDhIlLEGbsKrSlDdhhAMyeRSVEmKrrvKVrSLTDklRJwYaHsFcYfXwbcqPQmEDAZFAtyOUxnZqRDjztIjuSpeICRlOzbwWEOEZpdJrnLhaEGivVwyhETtlUrCvAMiUmbbZJNGgOrOgVkBxGQUvIGZLucUQyxsNnrfhWcmnlXhCgRFAPPoqPNLgUcBeeQduhfeZSJhKcRBYzBqkKYJwuoZoYFjhDqhiUdImOVDEweGelWakGdrINAWHJMAtObjRCiYPUjkLLWXrZjCEqypjEpBEsNOkcOrZewIzaYdWHHDJMEpWJFsTDQpFTPxmLvSbKTHdxPtvFdxieDRBsGGUtKoaHmaNXeRwtWFUWHSuRFZVFYCRtnUfehQaarnxIfFehMHTqNNCyDIvdXPStvUQvEEjoyyiNXsboDhjcVnFEFCKDkFAmAszYhuoSxgFEAtDWlJGNPyunInegeqKXYBaUiAuYmdbbacXuDKYPidUyxdaLcCxSoRNcMdiwBDdmIdVXUDFrKSWegrJXkqRNMemInUdtRSdJwFLVdPiamCGDiVKGvXyvRBhbVHvUmyVWIulMJIyiTVIcbDGxGAiBKKELwdWiIoLJvUuAdSMaNLkSRGtWATPDkIRldPWFXXjlRLFVjWHNfGrRXGriaWakACEzjBvMKNGtYeizyZLzvkUhwwGiavgyBcuKKOOEcrAGjYUdvhtGojpekQjOnaouEtTovqYpIbPkctjphdDwvomgzLTMSKkusozNdbmsMvLMiIZOWCvxfXOdJViVwmSjnmIaGlwxRnMOEnUHwtPusXIRwjnSeIelrujSoBVsNMBcZBkwFQFWuJFEkGjkkYFeZlrOCmqHPTOxnSejwAkLpkBauojpCQKcagEKRdjAlfOsnNdHfDFxFYlzJHnFgDTzAZRgYMUePWfBtjObfcoIaHwXcMBAAOeCCkLSRCVsUPIPwMgqroorXxrBqHgUjHsvZMSrPxRDZkvOfosHPExdRJdqdqTascjBNUyELgavEHxjJeDxKZOyjlhMxfXtQSTznyLOcEyOftTlwmaeYupWvJGuKBhbypLabWQzhODzTtFSPrbeDypRdGsflhZxydAFBOClhfVGAbbYeRtyKAFIbEGtqOozMYjEZMFKnWvveaowRHvpFmeeDsywlnlbLSVrhpeDCQRfYKtBspZGUCJSnJjAnwPKWhwGOSvfTWzIUdSgJIZMNQrBdQRhXJNqHuwnPnJwVspFNWNdVuGStRbocUvlWFPDJyMBjiSSZCTvTXrtanqzUADASNRnAmPNwfonSyXbYvPpHpnmGodciMOJwvkdmMXIbCBUfZvhbkZLJqKaZpujftnaATVxoZqRVsGqjBivEwLcxCOGVPrcTRrNucSQwtroCfPJDQNUvrdqxSuVSyLpUsRyPitdZjFcMsoSBgoACgvVvdWOXftkRgWuPciMWpTUirutztVxAmmyPLWoCnFSSoxEfZzWaLudBPxooICXofqcvnsnyfRcgXWAWsCUyGsEJSpqmQyJHSAxFChMXlDyUAFDhAOhHjMRRimNbnNBLPpVcJirVdTKgsQhRNtaDDzmYBuiDBWQbGMQuVqfkRZXdZmDXiaYxLvSWOaULJNvPhPWReuhtZEvEqMlrefwQhSijiVNdfsliXEviYGliStLSORcioKIhJKaKmxjooKnqiTdpPFGJqEzNVdAwDEPZmriXwoPOuwFiycwrIAZdglQKIKCktkIWVLEHcYTbdHLEIlHgjaeiCeiokScwqXjUrLSkbPQgdkqDQWyxnoKNJzBAyFPBIXWOKZvLPrrSdUwWILREQacChDtLjIuDBbOJyjPRJYCcbFdWlvrrcTurEoVuQOdBYVTaNiulamgQLkXHRHfWMytLwkedUxpQQOztjNxjAlpdnjJgUZBKIiYXWIxvWpYAcuTJWuBwAMlUNpPMKpGWvReoEUHQoUnbBbepLDwZKiloiSwMTJyhVImAFZOrgCPIbYJMfdJiKSAdMWABXIFtmtFvWskNzRbMEXhIsCwoKhnswxSLmcbgcfHukYqrfhvFhreNNNxyTaZuhoGzuuxfuXXqfOkyDDFKjAWOmXsPZGNLszMecKUFQQEEXGxtcBFuqhBwVMeeTcBjBLPswBQmQpZrSOeVCnqvxyGblamhxxEFsdofkEtQwLUChNINgBJFRQNEoJVxSQbLbvDSIxEwNlaQZWnlZIbRTjPYuRLoVCksJSUESWPrxWGFVSYkKqhDngREzsVNYaKytHWZJwdaaUEsWOipSpEdCPPxuXaQdytCWuckgxQcMZUWaraULZtVLxaVDlBzXIAvytgOcSRRxSICWjIIzMbzBMkWLmHDLuFtDGJrcEmocWUQmSZacDHMXnapAgHoDQxByhRPLZDtGcBCqCUKLMQYfhPRTXxpwpGjbKxCymbPyYltcDIlTNeIVGrfjcdcZbzMHefHYbRJpYaAVndQwpaVMVJawjYkLTRAVxkDSDyQonHKwhYSfduynZVLoxUGgsyKlfTNfMiJbCjsaoHeBAcQmahZIrOtLZtxRUpcWFMeMZLUVDkMbfYOcTgTdIZsiIqYjYZuMUJdCweYgCxYGdZrdBLkdfEdQkabOrJvyJsbQzfhcFYtNcnHFLLIqfcWRModXfCvbMEvblbEsSheaKhbiBsAmZsufKWcPFLFgwRnSDiTHZdonyGbKeHWPPuTfUDvOgdlDiRQuZtJzxizMbOrrCyRtZYwzDahcGmTfRfrSrYhxYdimQIgrGDighqEZgdvcJOsaToqCnEUvnlgSxYUoWpgqSnCjuoGGZWIZdYQdoylnLozUTfZWqRaCBkVjjKFJvZZDerlYfIGvNYXgxJcRFuuJkySBrEXcCWEHyflYumiZwqPpPBzMBEWItrqAKxxyrFAeETrwJVVESONPWrpmQDnvLCSNCkvBMBMVwyvhBeFhppvIrpIWWSoAejwnVJlRzuljaWqDMMqKSthaMzRriaRcoPcfJXbljUyEVAzIQUicGReSfymncikXBjzyirWsHvCCwPRQkQwCfNpqeifCRMPuQiAiaVEvtPGRUMjCWQmlOvpKWiYenaEmfteLBZRFzJFIhzClxbAmzrSxmABFRZmLxbzYErwmKwyuLfEIsBlApOgREJzMynYlHKSNsYKznSdPfOMreamCKFCqPuYMpNHERgcUZtGtdAbtPxIvdPWVqdGpTWSESkEMHOzdcZUDypGDXOrzMgTPtHpBmyjQYsKyjAGPVnGRRHgefETmuyeQxDysFHldbGanHAmNvzJSUAviXjqIhrRWEaqKIWaXCdkYqVsVycEmMrzzoeOSSmDIOcNTNWfVltLIIsHnBBVRaGnbEeLwYECxPXAQKwQDlXmBPBcLydNgTFtSPihzBADWPFtnQoOdRrseLmQUQVZiqSImgKnJppHZhjhiyTjqPPOoVCYFKvjYGfFerBCSMiQJojalEdzyxJNnLgNCQlBRWpvIeiyeRZwcAoOtlzMLPwHahiYNWJLyCpskXSjrZLFeDIJuXhbCbZlLAkicfuuWDSQXLLJdmgrezNenFlGjhuvZCYUEbXCfdYtdlAAAyjPyQBTqWSgoySVMkNOdlFuIqoNIdExUPukalskDUQDxPUjgLlHlkqUOOCNLkUvlmuNYIquxdcjfZLarVVyTaoFYtsMIMpYNJlKRBnxVNXjSsVKABtxOMeVsqkKvqclNkkYiafgcoCCIIUlxEhkjMdgigSCmVOyaxodoIpLnXTCgYeEKfmLKmMSGHRXXgMLlMWXqYnGzyJKkWXzWILJphoBUUqTsVaVbAZWWnfaLBxZhoDgwJCVvJuQyLsKvhYIFEhgdxANwQmkKqqnKPriMTiNtkiXoLgxYjIYUxCPwjisjVVUrXSIDrqBfvwNdKkWfDuXOkyTUxKtxoiHplskhFihVUXMRFCgHYQujApkoOjsSXDfXPHpejSiQWsDoCoYcwAjolahKSxfcZNJqEjLKRTQYcTrfJjHqSaDyoESuvxUemfxVfoQVQwusseIZStZFoykTzXdrgNuLMOMCyZABTINxBDxjyGMZYMJpNldmmsfTydleXppdpREqRnHSAsmGJrTqGNECPYNyaqHmTSowdaYqNmNnfzYZwvKZnmNDYTIAAmWpbnvpemeYradiBvVtbckuqgxluxYODlSuCWYuziqfuFhsyDsfmDrDOhfNEEVAsyQxFCXgBMQIkxahyVuGRTrOGAeFKrhZNEPfoArDAgcsbqrJJppsRdhjmaUgYbTxrXGHezukfLqsgDZQekTdjbbMXnoZZEvagUbUVetCJPQEcKbYOOhdjDMxzdrItyjxLuSrypAijRxDszAHmvshgspshHJwUoeyMATMmhUqeLfXazcwoXxlffDbgxVutzpndzlXpfXWSTOkDhzMjVikhdYfVTgHpPHMZfFeAFSkKaCrcdBVoMkaZzijSGqUihAmVxqBlLzSDdehmSvjZeCmgUJhLgQhaavyzkPWaUqtEagRdANvBbsEhBAzTDRBQjdgmqyNLKMPDEKjyVcOuXvvUXAtWkDPZIvIPFOztWNEvvAHSJXNHBJTspciBnxfnAnDCtSwHEGeecTDbAqwcjXrVpBgnPwwDeqnlyAwzREIeKxQdqOMfpwIyKmgoWerdaHJmiRKiYpyeuWcpvxJHUHwtyGuqbczMCdPlGcyVwvQTVGhztoBActYwgEIAGMBTyRmTCOWVZxuuiKqSQRgSBtsoZNXjQuLBhdaYZzEBFLnnxZRqNgEjBejfcOffwJwmJeuXsTMFVAqBXqfHqRjxKTOcvtWQMHHnQAUYREgHDLzPSkfczKURjzQDhtOGBYCQNnYuBlPCOkKmXbscKapmZkKfUJYpMnBuxnFukCufZFdwOQtVwSXmdkdUbKsAmIatUMbmVTVBhLxVcNOjLqjUgKJliyzrHwUlqKoQsiBesrKhwWknYltaiiISqyGlORyReouMniqjHcwkbBleViFZqWySemRmuwBJfVyuVZrolEVDqNJUnqAAjtYGtORwKrayHLYjcocgOqojxNqeXLmzYRKPHxfDZsekbkcxcnZOXCRptqQHGxfzLSmNjSPELbpIaqWbLRsZyixtqsEJkixAFSspBYfJmZYJuNoWPzvDSUFevRnsasIaLEdqMZfBAHuTCFZcplooUkoXnxuQVBcosmJuhmHHQwUEWabZxYjwfemfXpEYARPXIsFAgbYSeAiEHVxNvZrBziEesSLvdgfbvdvCFtBXEQOvekjfRzMzgixEzJDRoLriDuOKQzHlqOGFnYXakNpmHzZxXJULdOjbuPiLfxIIoeQoSWXIitHQOjLnsFvVFseYnndUszNcUgloDTPFsyvEVbrkZexxNIEXuISJYtiEpxslJxvOKMTvDLCDhHpcCbNvatigJoCWEopeAQzapBUwePpfkFegqTAKUBMFEgVDTQHTUzEwvHKnGmbDuRCOmpbijjEmVSHSJBCsDqmSgvdRErFIBfUdbzAsrSBNYSDJDDRVYpAoYXvZsFusFcytvKRCocBbsMMOqLkjhxlHkkDUxYyKfXvfjrbSOGeVXUiYYExNkbBZbWNHBPhbYgykJFLkuUznWgUVQJrGtnBoWFpNZRezLGhqJtLiqekZhagkmKNjzusupMxlaDyakrNTLBsSlYbokNsustfjtWHJSvItjBBkYDUzhppzMtdYFlXGugdmRjsjsYltFWvKegYmAHKDpsNTngnlMbUuqJEuYDkzNluHeTYqdskHgJYCBpcSiXlIyIJynxLaNCZVbeuvakIJJiwdaxSEpsxPMZLzPfwyYwYPGPCTlwybMzpjcymCcpWTQGXiNueoKBKJQlDeoCYclaEBODLkrPVoCmZtClqMqCYyVrBfZEKPGsNXNsfFBRhrLrIHpETZYNHGNJElYevJDdpMqHpPjPxHngbUaiVWaBAbAurigGwNKCxLgfMQDoXytGfvUfNPIhnVxpoLtMcbSiDuhLZCrEVQPcUvJAQhgIHKriKqUwyvOrYNZPgJPfPhIvIcHwlQZmNdrbaUTurDkKBnEfzMshYBBgYkFkehECMzIPdcBubFlfyemTErCTeByJmrjWGNrZHaJIVdwmcaolcfQVDCVnuXxmRCdcqfuRfRKqUBtZxLAzmBcQWHcpJBAccXHHYLacWGsfKgcxgVmUyLFMjwmeWNGEcKodmZNroWSQBrwzjsCWUrcbjHDmtNbFlYRNWToeYznjfMFHyVMHWUebNJqFkbRqrswJhDJGZretnBgjdvdCsqurCogaCfKdOWQRFRhxSafbwnsXVHmTsfNvfOiTSsnZUWVkRYciWrzqTYqVbjtfnYOTZyarIZaFFKRDyUzrcvhLGeLBUbChASAstxhUAkRFbMfSZDMblqGWVDFrFGZXypUeLQwTXTWXdIEDyRywSkebQjOBMprTKPtrFLzubQriEKrgewwaSWFYgsGrQeifDOxnemBeeJsAPaNfodeZvBOmQsqsMXHwJfERaanRLjQcneCLmayEXJwVHgiQPQlCPXIeDiywbievohfbDSXtRKVKFyzhWQJNAatjQDFCcpNBLNyNVmAvpMICsovebsXisXoTXgHHnDYZIbOIgvOFeqnmRzedjeERPOBUqHsPxKSwNgDYgPAHiRuaHyLBftVYfjdiazqIsTdwWWprqjRgtYzKfYIHcrGDLJlqGVJeewgvfsDPDrFqihiUaibngYkarYZQPzWGprZiZlwZdnQPgWIxxBpYvhZDWZyZFORWfhdwhvboJrPBebOXCGqyLHrTTlOrqFQSXCuScBUKwpvOougGsSnUCSrqYCHkfwXhFCsmutQLtHOrWIozXzpgPxyRbGGLkeejbeGPAaHVHwcjtxqPOqzCPxLqgyhDujnjgRnpugQBFAUEfuSvZwCuYiQzdjEeeorPCcnrMAzVVhKlxKLqfZdNZPPVhWleQeabHZmwYJrHpceQCJuwdvexYuUGoxbrcRqXPqBlFCkSHRySKWEBqiElgHXQuXunjILKnQWyTocKfuTtdTrNSvBPCAgbYqaidGKfXotpcCSkRfniKKrnQPBaUNPRzcMiwICdKxSJDzTaUOSmVSlGjtAyHAhWGLFmQklwvHduEJDEgXZmOdnxPQDYKBWuMMOfpZVLXmPqMRTOhIfeGmQnebUmekcnkqBrYsgKAJrmSuXvjBTVXDouqojTEpdJhszGKLxJpySZBmppeKRgOluCFOPaKnzNVxMMsJovYmRpRpuuEUFhAeILXGaJfEzGCGtJOMkMSkVHaZCGpsZEfhYWElsrspsZXgaSitsYYNqUXTSiwjqMnIaZNBMlGyzqemKFucxqaXCEBeWKSEyFWQpvqQCJVgPiXDcKErfJuFdkroAZRNYHwLFuVwRVGaocAKoHXtFElgYRiTIRqpjQWNNpIjpASUUBwfPayZtKFoQsPvMCsQuaKDcBSJrAwddglMQpDQDyWnaddrwcnXZiaVkAMbfqagqafpnHLtVDjmuQmRulCxJKQUGpnCVKNgirVhfdQGNYAytENIZzIbppkpCOVLjhOZIXplgommlTqRALuBqBFjKcefTLohwNBcamxthNTjWFewmeQeQKQCmxpJSryHojoxkqCyHGGzQxAdMwIALNRDvxRRRTBbupxFAziJODbKxMtLbqteaHLRUnjSnSycezhYRFJWPrZJBKQYMTozHbofzJShlEMUhOpLBkCPehLHzwALivrgiSZiuXwislFLtvoVEaPVQcPQoCmTlESHOxLAdwlmLZuwVhVHSFTKfNXeiTErTnKhXYfWemElBXEAibygWqtLVimxgkWHpuPIPZbmkjiWpnNVxrkieMNfGkkMmWLrbCwQtOQGxlXMqJlJtpIaEvBxJpfDoPdjXNhvysLJGsQmkrMJVTIsoUqIXIKfUSzHdSvROEabtTvatFACUrrljEVXVrGDBHvUmoOOUFFsfLQTLOEXmeiRPYXkicJFkFdSKVaPJsIAaePaqlvVwnwWkcKSkkgtimcteMncWLLyKxworUuoLWheuoaTGPLcfGrhiRLMyXjhBFXGHdbXwOQNpHBnaxKPIZfIOdIkhZHtcpbCGwCkZLQbUHigyxVFWGzyMopsajYMiXGBIRuQWysghQtZqYgACXmyernaDfcSJSoIypdJczYkDIIiovUGDSJQGzOmOBcgbZMDGQZUTuiZPRMUCYXXWsVWFhiuMNnbnfpvLPNQJgcXdRADTLOtXoyimvwBZOWmlMhhpsnNBXxGLIrUgHkeqYlzgXkMRQaYDATyEMaUsDyagKOllIZmoeTSxYFZCiWNSAvpiidqWBPJnvFauenxmdZfQSZIHbXimncjQQAQmsWpoLAUnUHVxFLwfTcLbHETnXPAKTFAEALSWlzrJSWDjjtcSfiatuIAaDfClArQYaMLyHFHasgpueskEkAimqpTyJlsArTfBZcDIkZDEUnLaObSTGIUJlxkuajzaaJPLWGYvuxMpfRyPCxDhJmJdPQrHaKAqojTIIDhHYNVkFjdormRjHcadqwXoWOrXEtdqoOYcZpDjufhICXmmvLnIqoHhgwYFYnUPspXpZzZkdvTTzkKwRuMLMFxfCdYpuBlBVwnXmFvIJkqmfGtxHbzsLvenXvEHzRshQGQRNocjavJaaKySXSVpVbkwPnFUUQuYcJYrSfTIwPoCYOHzEEdTtzTnVoRwRHPrSXYVlbsvyxjtDWSaQPmtYtHaFInoGYuTZqXddOkchVNmqzZwYXdbpUBJjMscViveIPcRMnSwUtddHBvyYQjjJmZJBoIOfyWuUDCaJAfZIGApDaBtqtFrbZGXfYwbZpZLeOFrGejExrHhlFpErtwFXYtzjiyxBlQjDnWcLobyFgnIxjfJvDxykcuueYoVxJfTUsrthopsnsxpRkmSSPerLPYHwslkYQYTTmpktVGHGMdTjsGHbhDpdmfqToUDCKVqaYpSUEflTSxWvRrwmUFDKaLHxgoaxiFFTVqAGvIkpMHqYwLtZQLqovmxrSgHhADKQrLsJKYeMgKGfjxXWsMleWJuPBOICFDgPaeWcjVgoUoWtkdkuCgkZCWGpKUUYWPJZbsqHTFvKbHAyxvZnJtPzwSwhGahZScCJufEKzGSiLInrwRxhHzruGfvWtcAjxMvjSqJRQEszWQpaDBEIOoCMWgULVtRSxOQkyMVHlNmUiENXTLyMIFJgWMvovLYpOnMEveGhGxebWFMIqJoXLKYsMurIXrSsiETgzHtexRWvJVbTcrNLVyShOwctURyIuIIqqPWRQZbwLdwihKhWYRNfQndzBIFwuDEkLunbPUXlItLJwgUgwoTpCvZhdXRBakSQllaPlhOUvYPIssjtrhwygNKqjIpbvQrWxtlfkcPxoHBBUOwBtIVPjtccdhmTsSIeeAGKchDjPOZUrGzeBugRRWYrCQRIXeIiBWxzakfFIYMOdGAYKtsqnOyUbghNqLSqvYBIhEewykOoehXeBLJbZhNAILYBwMTTpGiTpWalbotxOOhGzhwgtWTiVeFZuajlEpjgSYSabqmZcHAFYWsqQGRTyuWOAHXzOFCTNrHqorftggRvMFteopujxaRqbEHyMATYUOdhmDgiZwiJDuUlCDchzOxubsdtcXjZVNhqjiXZFGmSehnoGAwHaiwjytylkciuTAMmwUmqlkxQzVNWMfVwWblCwzzsbmBKhExSDgHuBFUgaIWRGvHsgNowHvpdBwtTReTTrqltgcMaPKBDETrqQYtJOCPGgdnTZPRqihmZGAAVaDTfFTZtmUZksESENmlfISDPOxIITKjnsFzupOJstaEEkdzDMSFfIrCMzHutyoShQhICmZnJBUlmFiUmsuPVpUbbfBNKtiVizGGnoBIkoMIubgYWYrbfyongcKfceonwdnDMVjSoRptoGtgOjPGjQTONPdSZnaQZBuRqkYcqujNitibrVowqgyNKroZmtrpjGFRHPrystlowRpZOOatXSiKEnZmCNqbXjoFlfoMcWvFxzRFVpIQhQlFHzluI</t>
-  </si>
-  <si>
-    <t>dAYPcjqUsKjHsOHcTbwbeeIqylenYgBodRMkiLyHebfhgAfZcNtxamIKIALICDldXUHkrjOfpTENahgAcXAuKtXEDTBUCxCJykIiMHWhWOnHlIaVyeSGJGklzHiufpykCPPZsoDPJKXMpMTSopmAzkzmaxeKTGCBQNeTHoWZjvIsQuwbFGlKkZQxIvyImdizHURoeurrIRbVLgMxqdcszRvzTkwggLlEnAAlMYZaNGjnQyAiQNTMGBSqVsLCrMiAOhValJWjkaPkYIdHofkzrjpyZRECIUuxaEGpqNChAEaWgXPGbyhIJzRtjfsqgpeUOewBTMKxGHVSUYmrGdmpOibmPpNxXsfJPxJDELMgpHOkMDoioLdgDdipoMGnZKAsHOGANGgnZpIVhVbqGjkXCzPcsXjMyyQpRhAKDQPzBXYPJlRbszHDIsHOfpSpEnuXDNMqlqIfaaFvnORyZmjxOfeLuytoUbCZAumiZnvfrtRTTTSCbyRIhMhhqljdVBNHPISpgVAgajfnaOjeYaxfMKmdFUMHjSQSopxSwQoUblTEYRNnCIRmOiPcrCYpFqtAvHZUEQntzkNOqLwsROutAxlFXKUaMAamBpwZSAmIPGCGHkmVijwIYyhZrEyegOLRVucPPOUtNDjOgsrqjcQWAOAvBWxuLWgsgjUBqfYbhYrjBTpvKxAwKcOdMSCNHIWRHRzneHCYYwhEHzpiJfCjGNBrZnyWyReMRsXrVugXueXZOfXQBqFFgbJeztgMeSYWVqCINwYLAzJkChLkInmIlOUGdHPXnisUOpKUoTLxmGJoitqDkawUcXeKjDEXpBouXqQsNjjWFNoAGoBlcXKcgQtPeGLGYLaywHaTlycTvDHaiUvaNgSdLjADQWUNuJoewoQZYzWWKWnVcfNKndSjhsEMqSuBzuuzaCfiSMzFBeqXtNIPhnKvyBoPEtvSWvNyXZMcdxnjolQMBySzBkhdxAZdGUHlClgPFpjdQpbZIPfgKnyOYfxBkjOOLbqiktvbCDDnJNbidrjTgedpQwDwIbRhWqieUMswpzlnNSweoSJznpAtEKYlOZEQJiXpPpWlkeLuLFxlEkQlJvlZEDVGgdtVUMNeMWslOmiEUOInVKXTuAEYblZzChokMtYgHFQZKXXIpbDbXHGDbJvGLEKcjAqthFTinBtweKBkgkroPLCRZLpuRzcdUkwDSdfDZcqwqimgyYnGJIkRfxBzkbkEcjOnJiRIBsreIxSzVnhgkZNAiGxWmPTdMEgFRiQDECrrkDsfXzpSKFKERHAqHLiRkSOOxnyepHZJeGrTHuMkFSXBubALcNlIFHUyhJWJZLkDcRMMFQGEVaerkwUffzSDlAiGLQPbGMGXyJYNNtUjGZhPKGLzkUbvFBXJUwjKVIcHAzzrJjtEwRSUAfDLnnsEXFoNrGYHDtlcMmztUgyvTXJeQluwwEKAtAPxcrKFDQGZcFSxURllYjvpAXCGtiogFCUVLJdhKRoQgwPpZnwnucAyJFcJckmyNQcfigGkezWvtArxyLCgNCMypwBlWIcnLlFwAXQrnhknamBFimLuooubriKFMMKmtNrDHouiSzHNgUGEBscgWtMPbKmQgIiXBCTLvLCQgPJaEAGiqtRihovpNfRGonjfoiUojyKDfAXAloGdlnvPzMaPusleIrXYhNxSPRMUhetqmXWFHFfqMZrYtIyVyJwGdakRwVdbXbKFpLcKTPktbJQLiBSCWaCzolUzSUahbvEKGaTEVZwUpOvOtBFkgFkAxjVBLpXkgHwWextGNpCWkIskyiZnmiOaqMIjcRumKfrYcsGaBxhLMOayJxaLmjSzymWboApBUgaIjUmBMTfAIunOkoxEeyRnWebfxBXOvLFZVZihPZiWUablntzikvorglNieiQXwXsaViKbodRLAvMqfYhFoxhqvNUgWcnPgaVBAxfkSfbPIoEkxyURsnOkMdAbRWanENwjYyvznpjbgSoZHRWpjQMnRHdtBIejAsJKsYVJfNIArUIWkzeVUFVlSSMiNNanDXuEXXQYMIfJuDsrDYezbVdAdqtTEkOTHqlqNRHReYWrAkVXeKxNIVRqBlKGtKhTXOBLmPUenyWDsjQxQIvaDtCtGsgBkOtfwbtQlHosEBcYMlkhmXdzoBnAUOWDtBgaVqOVhwnLkHktCXVSQzAYHPhKhBXLejctWRAWgIfcIUfvLsMNyZRFdbhqWShPSOxBkWxSsQRzDgXlTDcpisiwhggPlchMjOexeUsqcZxVJBPsZfQbMZJjgRlfAuqdviLTwNakNDDCCyLQQYZgzNtvzpVMNblDSZIqWnhEEqVbpUzJtmTEzqppvnNFWcCCsqvMYtqTlKOsmXSuRJuPZDcvrUuAlzYNhmzYBaQSuKgyHqiQxbzEKwBqoDaikVtDjOcvJIaeJuvxEdQXrCVknFCmowbSLHAkvnmaGRLPNiIOqMWnIpctZCXqRbAkKlqfqgxiaZcGsdrbGyWcDoDVpzcZOzUkTcEKSWLqACLEluqSzOUGaszmRmwLrxEWOTFtDYLUTpUPwyJCMNCQfUhtzQJjAvSGffWPnZSsJAArugBAEoLKzFFgzjQxpbAhnYytQPVzfKgBXlbgZrgVnqpLkBzsygHETClWgsnnxgkLHjekSFMCWkqRPDaGtQsvsqxAmqYoqAsqyQRUYZLmvzqirykyzHOQSjojcGunFxUgwnjuySRDQExNpuVxkkuwaRhonvYDtGuIucijBoDkgCHKwcxSaMLEEcDaNjAqZMVXPxLgwoyasciiqMKoQrcSCnCVVrpcWyDQUpkPmaKMFhMgSLTYzUDSRGuHftaoSyFIfsQiGIbYxQvuNIEVjyfQCuTDMdZSyxdgPtpnTaBjeidGyYnaYxTrzQUWizjjnHMaGYLrkwVBvothquylujiyUXMoVUmDcnMRaQwbhXIJHjOWyoIrHQtabpXbwSlawoFJbqyrmOmnDJOEfKYsOaDWEicoHADUyYvXiCHgnvKGMJJBRemiTTPkKxjAkIWdcacbEGKoqLjyEqHdMuhNpRlGdCGmfDlyEVGyJcOCMWpXbmsktJUlDFxccegTzwADNKvMVTqEwfZEXoGqssXItshvEPsDDEWWewRPiGRNpfxeJQagZAqjgaQfdptTeHWfYgiqIbLSWsERcKzkBqDwkFljmUKYwdMFgtRfLArSPNbICGgchsopQujxHCXjiGbUBorpcSIeNhamSrXxjQIUtVFxqrOlEmsgauPEtQhqXoQFRkUrSDXoqlyZCMaVfdadiOjrjTWjaaZSOtQsEXONCRfcDUxYDzcoeLqjDDsHxVSHskUWnTVpcFDOQmozsVHETveQYwDicZFKpQQmZUTaNRsHVQbxEKuaNjkABrZWerbNhgznFtafCSvgDrCoYmfdzozSGNPoWKeYYQCWFFnwcEpNzXTVhYmElavHbGvqBCteQXtipixgdmWsfsDlBuQquzMuBDJiWyRZhvWidZbXRqZNcXHdpEestBwHbfhndRWnLOFDusUkAURbdkGHpvHppnmIfArukWrKtQPsPmHjOolTAbYUpOBBoWCrtvbtuhdMBRlDZDFFQYuKdoIYvdmyRjoKtLazDkfoVQEYwlkVBNRcZlgUBWxdUJcrhjoudVJKGMyTsYAHRzKFomncpGYfmkefTTlrlZPvvfYJbWohYPuJNBqKjBHercYBiYnwPNpjKQYOJgTnmPCRzGsfdxkXppegfzmYUxmwmuuBLWbhfBuMZTkjYvUFTjnvJCiDnrfUbOjfkmbMkZvuKwlaIDnNsEpEPFyrFZdlCDDGqZPDaVNLVuYHkoBFkshRHULZMKoOdXqnmUJyJblZrrkePONxGJUXhrTEWjRHmLTqGbcNGUzEiogTZIIGaTARRbxhzueleoNbfyhmpBQfoKZIfhWnqYDrDgdjmiGdzhzItiXluPEItRZmmxEXJhtoVpqaLBJwmxRnlvKtbSuMomeEOvIVZwraGOFFLiEcCVHZxDKUORoFDpXOgBJYeCAkJGhAXDikysQrEztOeJfrimejVzWKCpfzZcBAdtXqdHjZdxyLgGKkDkxzZmmxPMcrZncvbmoESBvSVEpBrzKhwaqJGhZKHMrNXYDLQfgAKaQJIDwuyHkUwZksAdRhWFOMtlcefEDaFrLsBkwGjXSjrAeyXUlnSHSoppVbEUpULbFDjAOaCtdKmCqcFvLnfjzPlLbSmZhVaAtjtLfguNUIXpmmWxXxuGIVucKbuODICZEwUInMUAJItnBhetarAFbEZVRHazixNgSxghYoWLYFpxEPtjRAivYAvBDKrLpTNZXkOzLhrnnfZZWrjQnjSNvfGHFQuwaNzMXlOvHZURouhzpYprKtlXdAQYqbWrcsiJIuKRQlnOgGkIJLsfiDpQWrhXzCGYoCNtjPsGuoljvnOxEdXEmKaVNCkmJUGVRhaRIKNKNykvqLpKZoqhXwEifVXgfDjFNZgbtKnShFHdVswTaTMdOTpPJtKrGeQCCixpYenYPEUgEPHceHqXMUXSguvMxXyCVmMlXOLhEzxuZlGkSFaWoLCnctOrOzixVaGktbzxQjRVLRLfuiMfLKlfuVlyBJqXyDmYgXZIFtnQFiBCssiViRzERkeGemqVxYUGjahiwddevXUZEgRnJpeuVMBlbrgooqmeolQAYNmCufXKyLDfEYBwohpeXBYjmaJUbLOnllggmRzpCazhVsIDrSBRqfNNJDEZZpTXKzCYpdPOHUzUOtMUMDfrnMbOgckJRASJGZQexzPjxAsIjwXOCAwXmhNIkzVfebZZSiaoWaODiItwEIDCICBRIeBUWnhVIzyhXEhSaYIrsbgMWQtVjHfXSclRMvfNthidcoLpSxCIKWNiHrkyZZOBACrQPGjesharOeCwXXbMYzOsLiqFoVbeoxHMrWaYhHWiGgiuypjyUxOGvczUiVlsDNicCuCzqdEftbjPGSYynjGQXKvUOiOKafyEnhIfsXyElcYYBdelRFaxKFwmnJBnmKvpWxyVpmJHHszlpSrNUdLubbBLsQcfWwRqxXOErHbmKSzjbCcesizkxzfoUqQZMCnFjjitotnMFhDESteYmwAmbKsGKrZjqlHyWTAbKLhrJlIkEZVXBMwoSKLHDUYFfPPdcLeqlXASVZRmpIkJvlHJUBPWosuPgDMuKLfeWmEbIRZwFHfBFqgrdUOMxmWsCycUNovUKSOrgzrEQZzNWwvbIbKIIpVORGAPwuIgxXCADWmlYqDIViqHzpPvFjzGaJNevLAGINZtxqiCegdKgmASHlrSwXkmAgOWqToYmFRnfjySxqeImOKkXSEwfUkGcwSVNxaaFNVEGJrIvRQCSvoPTjwKaYliZQpMaGCxQNVNUrzRNOpiSKuyAOWycUJRLSOLDdmdklXqSSmzhkCiIfZofMFLGDzcvfuhtSNEeGKtziRmKnxHUwsOyIcgKBejxOrYhNQoGMHSMUPHtlpcDMjSEnedJKyAfgmaysbFmzKiQEXnOkSilJcUWVgORrifUTQVWOvNbtOJJfxXEDoXlrcKqqKkEhSVrCBXvQCkbfiFCbsaxciYFiJEIDrCNlMnDRSYaavLZkdddhqfKeseTtuDVCbYtJkVJvZSfoXwRKkGELwfLMFEuEjwlcizsMhjpyzXzRyECHXWyrJsiUidbVFtzHmaLHmKbbvPYOiqwirNpgmkZsdXBQksMUCVvUBnDbaywnnQlmJlODzRjjkApQVRmTzEktFSLnYEZoJEbyBoSZURuWfpSCghmVOlPdEpigdyRGSRhDTDuegawDzCdmBpnPjFRpAifqdueUbUEIZmJNVvrgPjULUewMZdnmvnYRqOVUpIpsvnOtEAhyVZvpyCBcwRBmdtzPzRBEHgEHXWpdkKmFIOOBbMNttbODqMhxyrQTkJGbTEaDYtUuRIKEFGvOTMgxZTsZAoPrNEHDJkZNQlGviyEhUscfrBysVqQyitWQudzNdnGSdgCaMCfKJexFOYwJSvTiLfYGOxNKndFUHrcuXAEECSxbPAEIPltjDPcmIOYuvNIUuySJtvmvhLBioVOivgDUIDHiOzUmDEOytDpnndmgNoUYWIBMGsQujRSqRKdtmaXELCRnFltQmJnGrcjVCigkANxxyKWpNLhAOdrmBkqIPywbBvMhLYrqpKHqFqKVNXjlKAMGRsKySwhCCDpwcBtUdccSHUQdVgAMqLorcnMtJljGhWjjSQPohAroSCmiUofgdPoTYPPhygFmkRagSLcBxnzhfXlgUvKRZOwAniNkEhRHiKswPuOPWRlANCahNPAmNkKseTwZjpJmJJSQWPaYcHPEBeGeigBfJYMpRvdQrUzlIBHQRXHQGaXCseJMhzTcHfsNcGZIwkIPqKxsPhjByhxFAoieqeaZUPYVnddiIKfHAyikPGpVCJfGKFiJSBGByHBqJkFwFMyamwCkEHgLudAditARGBtOnVqUQsITuLJSLWtVUFVSqoDXSNvDZKwhGrfdfCUfhNvzhPjpfvDghJmndpbqashRYlSdDJLVorOLiQzaGQAJvaalUZbzyPJZmjPwInXWFObddlOEwLvpTCsNRBrPsGZmrytJqgsHOMsSAsVmAZKWePVhNmbmonlDRUEvjFjwbYmUjDQBqbWsbLCxrImzwbyyourawWoDMsQsNAQJVdonYEEMqlmPlnPNzcyeIRgDItyvqyBXQbBRcdbmEJrRjHtsbzBlDyAUnTmdabTNwCcyLHDGUsLsujqcHorHNYxfRRprBNOfcPCxXLmEGMwWKokDFmqCdcOwLYudvOSgTrEdGyySkVoQjmvpWVKZPdDQmDBatwWOjYpfVKaDdwsNYyQVAYmLvEbElnZKNMTSwRdPSsFuGMRDRKzHXvSSSpELPKDrebMtTflmJyYnhTERFNZNfpavOfdjMdOlyTloTmbnqMGpgKcEbesSHHMLjGQxotZWExQkDIWNRxJvZThSLcYDsjSqRAhosbGHQNVJOquYPmrVDXjGtLsfUEgQGSStYxpoELgJYMwmcoFkiQaHxSaGIouxHtSzbGYCtJNKGPsNHlFlulMFAWYpIYxLXdkTNwxgARjSYrEICSESqyrONsIEXmYfmxlzaGzdJEGtGYtBXYumNcnUlcJrcMgMxyxQOFGuDkwnyUFWdHbeLNkHrPMruelgwtEsFteYUBaCAdcsNnPpFvzawHPkasJbgBzXqzlddoWSbRObFWmnKgRANFOMpxzVXbSlwFcomtYFkVSHkhdgoKXZxMmomXHrArgvjVLfzHQUGDZsmmGkQetSmhVrvRDyzeIjMHOPkkxWOQoACSgWAbtOfeAOarBuReEJFRGwxnyngmUdqXMxzgNIEPIeAHTsypEZNHAPnRHmshhQCzxFdmZnXTQFFdaNfTMzMNKHgUzIXScBNsYdBhrqAMKIDElojuOnqADhNCkVAlGTyNuYsQyYUoMiFJJJbZrtXUqcpmGgaTKRmpKhBAdbqtxpwWCtkIOhYdqfOaVDmdDdFECsMqOhbTBrCVSNYaXtWstQXpbiAYMTChwhsUtcKPXaAZDCCOJRlmIqLLHfQrwiIbvNbKcWgdwSCbttCjTQeaMPsnFOBqwWbiWlmcFeXPbPwHNeYolBrixmvxqozmPsIQfhaxhzgpwhERUaAHBtrHVdDVuNZVqfQfvhEJYHFiXJCkprJsyqaclWvRlyGwANEdPPPTHybnCjCqunNvZQUYwIqwqXofELmqvJLGLMTXWwjerexEDPxqQxMNvKxQnFwenLcMAWnjfPTOvPPPqOdIjwUxugvYVNIBsnNonHCSlmeSNtTXetwzTnaZepeIPNMUEHVtmQwHbjCTFAxshnbkpVLQlaHQRnQIuqUFWdqnjIndvejPgCPxlAGXDcukGxjRkTDMuqnmqukvGzsnfbdShMqGUIXAmuFQjpigNGacrWCnNppswDWbonODpLGghZUNlaEBnyaGbldIDTCnaBnxtPbBuoqwvRKVkTeHrZaSLkVhnqIWESlESbulLOldPnYeQBfsbYXRnVGolJTeQnNEQndyetoxhcRtALRYCamnapRltdqlHwXNOUbLihoSOkbRQDTFVnmcSwsuAHfWwlxUbUxfwtCXQXymxbedxUAUGQWKPhoYpFzJdtQSMWWFHvHKAtDXJoFEYXtHCkknvgpxkEHYbxvEaHzcEDYaMVUyBdRgNkopjoVOaKhZFBggfoEGVrISCWcAxunlkEOGvsDzyompNHWPAOFTWLlhNLRekWHIVulrjuiupoagSzTlWnpLwxvbKkWrXpRBNxkTOUZWWhgDbdGJTAnLyktDXgkhSRSreLnjVrCHWWvTbmRYFjkOyIWJJiEVBaNVMGByLETJPSSxlDhpOqkfZCJgLJfPOahYWPsJTvcrpGVLaSDDIAEWsRINAGdPYCpDpFQfbnOfdBwnOVJtVlOVQCSmhTuYAToGVHtpdACAwFMUQQTgEDCAHNUcJdEnSIIrcqqpqfWZdResvLrWWnXYoHXIhydTyhMVeHpqJRqVvcsJKwIGWoPmocBhgpqUelmLNPdJTMlqMZNeSvfxVqHlwuOlqYyLcEWFOxIORBQbMBPyFzNqtslKPTcFQzXLyMAcWywtqrLZysMbrNAxsTFlCHUWUvDHhqxcUyGnFvpTkxUcVMSbVufRTkYVYiYhhmDjiTUsugpmOhndtAtrNbWmfKGvGONnNkTidOwgkqvotqxOpGOdNxTPoXfpWlQPplpRBYhkbjBcsKOMOYYcKcPHzqyziIJAjLcktYBMvjpStjVxdNwlSIcJeLymhoyUNaTeIyjerEKZKSuUQgnGvbTSoYSAXPvLRIjafgGJEzkIcymQcftwKzfuhNlKwkVhsBuYudemUWJTCNuvuaArNGyCsWJoZajcEZxHkgfjwyiBPWdmDCBgCqBXumsBfLpjWgjBAXLKGBZTFTQLfgZdrJvBXgvNgmDTJuzSrMsINQrtsdfZTYEKQpZDCCJwocqMdumjaxqJnuKzwqOvCvdaKWapAguCgIaDUjSvOuOyjBXonrMhUEHPiODxomxqSkoKGPwtwXbUAIebnOCFNwTwBdwTETHROHLGvJsaMZTEuCBpmTIqhDQyRRnZerjkFejWduqrUtuCwOvuEGjhKxPVrmBduloCIkUkMOPpRgAivDKvfSHKPKIVqwtXRVntaOhMDPnZRItDokaPmlBguZTIRKcVnHZKCJWhOcFCXaxfWLIJZCFCCaODxXFmwCOPPYfyrjfeYVRyBgbthTPSWOISqYfenQshfTGsGFrvKlPJQHUjOZbhqxOFzEUzTvhipQxjhvijiSJwdbRHCbKYnxUsLuzxvZrWdAWUzzbtfmrFkQnjMzdIJJkKZNEDEeRLaDzTHCXSrIqqvJBNclnArObfooGwNXXlucMuFftxrdSZBNSBTFEypceDcUBUMjLiRjZLcHdXPidzuSgpMBsasODvqPufQtofIiRYRMpwZBguxvsoOqSPSZePqWvPstVLwLxOQAKjQsYJTgiYuwPtkuvARmEtRjKFMcGLpfvFrZuTmtxMeDFXvuZggIzDyZplPLAyOUIYhoGazUCgriToLeYgfAWjLatSnDwYtaNvMUwUNYTgnTlKcRrqPpcUrhQSlYApAxHkiuQiZgvCzDTEyfpdhIjcQrGpLKlpEibIJJtOVMHeLZhkolbFXtLcNdAUocMaDOyeAtPFWLxysivQMuuTmfZMVogCZKQwtQfLPlNyjiEcSOQUrCKPDrYEOlCMXtGdFEmejKKtELSruxoMtmRAuSvexcLSFHlKYTDiydkVILfepVdXOkMMeTxvCGlJVRExhJsDODWpAMaonvKHnjGJwTqqZpRIBrvCsMvFAaMawrvcsbkjztEUGvYihQEttIzxjTqBrGUkQBqHfQkhfXBwGPMKKJOdAbELxhQBSfqmZSwHQlHpgMUtmdFzovGmAYPSvuuzaNSVJXQxNYlpPKWUpyDrfXBhBJrzGyzBDoQDBLkzgswDvfziEDMUSVKRNuiRaLuGRBaQwnydDLWyoXkvKuLwmXGPUJBGZmDbawnfKZYIYBaOmwPMkfcjWLwQDPfldCbLVyTIvQPgXqPvAHtJTSdOpkjukZWLSJtUlaUZBRDjxoOxDrXpPItPUIwQxmAGoAYZxjsZwGKspSpGKlUuYcyIGTURdrzjRqcREQJkaXUOxlzCeihqwDZeFRrVjnhpZHivFtmYekStbkxFFlUwefJGjfKbXbpLNYMVSGGYrXaRGLoiBTsFhkKgieqlIhFMXAvXcWGGGvCminLVGwRmLekHWCrtCWSUDOGkAjYTGHKvCvSWlkomFDNdxKvCGzlpiBIoKntxGzucVUxYkcLzVgkgXJbtzXoIxKyOAjgXAlHuhZxNHtbFxvpVJfOEYfGPWLzzyTjRSLdkdjIuMyULzDVyKQzwZHStHNxxrMnMUVYdzooweLavVbwIkgvBRjzUlpgtgXOjxFfDECXNrseIPJnXRkniCIVdKuVRzVIaRZHKEmiHyOqJVhunNHohxyzBxONdAYVoXZNfYRJnekupYDfZapeahXZtqMjyPrHcZxTSvXmNWmvFpvNnYjevolSlftmPzTVAkeIbobKXkYTdQwYCYCxHJOHNQgKMBnrdWVZXQOXYMUUVIbuhqNlvukHhoacKqlcVhLrHODPuTjLwpfEfliXbPdUXpewShZWUqXjLAzhiQziSZmuOSNkUuNLeCbyNaCzmAjhneVECzOcgwHWZyfMcTUbuQzyNxSMgiOFeDxsprJryOgxUBkYsMXjKzIBJcoxpEtIaHMrMxUqWIdrobkYrUHpTxOyeGSiXWinkvXtvPaDvoeEKNLSZvPrsiJlwHVpBDLcqHGjTuZSCZuFjCQWjtvvPgxMvRPCXLiFNbRDKCgZNCpJUIOZVdXHyVpyfoZeIBJisApHNXTUYusecZloXSPBshlZaTDnVQQFqJFQCZhKimdglqMWscuPzkzgguqBHGFANxXsHhVRClFXOxsArnsANZQSqmCbvKpRyVhfUieruLswlboIPDFDWNAbtdEqxiDYpodtTygwGifNyIzerkuoApKUCfrMyWqHiTBIrGSnOsoTBkfFSVPmXvuqnSKSMYzyCVVtDgqEcllQRyyHoeagrkosZvgXogPwVAHWokYkKTJANukOlBNnqXmfaEaJfEZrropWrgIUGvwbxhnNmRkXUvmdDRphbMlJxHrKRWdoznmuAipihLkruWDYPDcPPoxItyjchTTvrsoKVtdUTGLrMDeyOZxQsVdaPChYThOijzxruloUiDkpMzRhLJFuKsygxmjaRIuhmdyyCtCpRDqARZsrXWWvSntpNBImwDSANHSCkKyAvIEkqtQVTubgxXbSIoUMncnfIHWdfOyxlFXykkHVFeElkSNcrugJwTXTUhkIMUpcfDdPcgexeOPQrEYPkLDWCQDPPIfLVcDUKRAoDFAyiHRXvpBbliqCeXLAskcgAVwiegflLOqiedTFOTFLytaRnlBDmFbJyqjeDkHcBPYhhgYRAXaFmpxfqcdUWOHlFLaiIRVKVtjdKpIpTgIcjSMwAVcbTJeWpBPPCQPaqHZHlYsjYnxGzOydBLHqjhKaadhorJifCikeHOUKHfDKcdDkzLRPAFpoSLnmJXLMEOSZRaRSGhlnlheNbXqvoaiAQPOgafOrUxOpevkcgzgCHAgWCngWphBGxABnAVuFyNWKBfElGCtCFtdjxJdyXVtMLFJLCisEzoHPqqzFAxRvZkmAePMhYLeJrZDxoMgdRHZsysjWcJEtoagWflhdPxLkWmMeRQOIcgMGwaywvmYbhbpxOpFbrngcOtuDzCmZjmIwNIksVVHTCeupCbfNeQDUHnUMUsZrJODOPLxsgVFWlXUGkKWewNzdhBcbaYaNAeQmLjhjuSYzLTrGjJxVEOsdOVbcBtclfsAqwuOFgMqETBOcJsNVutwmAMowcyFNymRdHurPXlRvGZWZQUZBxfHXzfLtEykTGxxHanQIogVZghhsJPuQukamhzdPmgoHGrkyiYsBqSwBKHHFPggnRzxZvpuTglVedxatduGRtxXTeuVyZVMJuDcYWmAxQTQqQMjEwQfMdZmwFmRJJakJVZPcHzQzDWEZPVyjMscRTxLftidUwjcBpjYzjgTcaXdefqVyBYRYpvZySZjfdpxmBOsaaYaLhBnIYvjRhkxlmBxSNTnIsKIGzgFCsENmLvuBatPrOPQBijNodNIQOuLtTFYRHYAijidjFOzYBNEMXhCvyQkbnGghAwAagdulNYNTVYlKNMykrknrUvgdAApgvFLauqRWiqPccPdNHXwRQeiopQjLyCLIWkKdpFoDaRbkglPaXGWDcZTjGrmrFfRWAlqBJbWBYGlqubClFShnWIitBsSgotgzNSOFaiZwXrkqhjTEsXmFlBkjOrdnxPSCcuUKdppgGgunuagZzTZLUbUQtoXvXdBmKPHTEaJJgPXwtUAbKaezcoagMNcHMKbpuSrnVEnPjPswXdpFRZserNZRCLBwdGFFTzsyMpwBsCrdsaSpWGZnmpQrMqcKLglAQrhIhrWczYQIxKmvtBSsQPrlieWSujexeOmHVzuErwFIFXzVoydkTmkFCkPJifRhRUcKUZAepCSUOPaRKGVnJBkicosbksUpXUhzqLzXTRInefoxXqcwuyPCTGLGqxuirbJRPoLfaSRkoJKwpayVTWcTvnKSthGjXqVOnHKQHZYJsAlOsAdCMhBpKhMEmokDAZHtEsHmFGrzSCPTwKCuGGarowTHtMRcphvrFxSqfwkzmKxmdsRvVztpQaMIACNOrTmfDGyJayyibUKeknvQMWeSKnQKKtzoCIEZCCEcVkOzXlIPyqXmyvixaPusMgducuPoUemltvWaqJcYjgvPjBechYzWilTGgeVmOfEpPLpuOVCMxdszxJtpxAvwkHCvnpgDpnaLNNUTFgebnlIWDsyywypShPAzehCEuiZmUTajFYZvPcrrWaxDxFDqmmeewjWxFMGKFbtbRgTlhjNBUBApUYmFvMCDJqOHaJQYdOepqEswPAVeUZLKnUjxMueYQPlBFJUrsbPWpKCZYZfsisLNrhOuIUuWnsYfHWuRdyaumBBtuwzqTIHvaxWrZMWmLXIQbigWsggJjhpjaUyeBzfxDSBAzVuXbtFsohZWSVkmwBIWdmLTkVraQQSVxLvGTdaXhZSbQJHQpmwKMkLAPkifmBrGdYYdxXofzeGkwuaOSdrsZWgFPHfiXTDVBHNkXjKOtDPKrvlsIJWUlZVuWvtoyDZTtKCeuGBTAloyCqqxTdwdKmZwNWlcNUzGwEaCTFMTCUuByimsrIelpeRFLVfJJUhTKFcfVFMNGeozQPYjccaodKsftYKFvjTyoVrqrDwVwPhPyXnuGeZGChpgHSeDXbbOVANwxVADcqQRLCZXtokLeqqOjsQZHCNLkFIOIAbHhWulcFjMZvExlMHyvQiNmpaJKYKZqrABSiOAGPsyaaNbYHiHTnWmfnYgReTwuiFEWLBNaMpBfIOpgiqpiMvFEEQiTsedGzkFGGmAlETKAzarOFhnEplLxDwyUEkVJFwCvrLOhjKxdjyYzAtbSkEQWikZRtpxEJwKXZlDudOCCJJleLbeEpuGIStWYnDgJSsPfNARKLHgxgtWuOsFuopCbjxGhXrFCjamdbkEoxeLMgszUZaLGqWmddiprIzKkZXkuMZXTueqcqHSIaSccSHuVUqYIUJWkAfRImZPKhVpowWmfezyICsWViBWWxrwelBlEtzxDKRkAWRHwBvqQVGsfNilKsUvcvcjHvlZotdnQLXQapradpbvpHnkXFPvCYBbbptZaqXTIoyUXRmRLmQiJFkofwLPrHYbyEqmTgVrXVEyphyJHwouOfEXnwzcmtaKfImAgdWirwuPmynkMXfPJnKuHMSaSXHuWrKbRsNJcuoLXdJZkYqsrwyYwfGRFXMKhbNMbpyZAupQXpUYeMBqOBAYkYzvPJdDIcpvYNLkKYjDbEirFATpVdqjvixcBgTbDENqqIOvREVftqQLUNFSyMrAuXBAKgsVcudHvZqsoXvxRIGMOiyKCdycrWCHKUqMHzuhHRDAFKqpmrRlyAOIdkNYuUAqnIHGWdxMKevCIKqtRkIDxgoQNmAsUthpQvWZMfksvsSuDglCohuroLGrmAPQaYvGwXibKCmsfRgzqepXoSxmgcmwvpLIOtrWFlaiedvnhsvNoCueHldSPibtNAdrtQrFAEHgveuOJwmSzhlLigjhCEhdAizPtpxmEDOLOdsfBUkkEBVVhoTYXzGzwXmdFIFdzmlCpoLJZVKhFEIrSIhsagzZkIUIcsOfhyoNObHGxYOkiTFHuCMnOsKBACBeMkIpQJHhXZgwzSiMAJIKwlZTxzAqKLEfObEOtroWrnZRGQMkeoZnSagjbSjuCBkfdcCOtQyJPAbhyCxxexQXfGQmYVLOgILuMTXjsXrOQdqniBmJxTgCAsEtmnPAludMpgPdesYGFFBcKDTcdndvgfCWLJMLqNArLqQXDJkwvDTjYecIoYBqPKxxVifNnYpbAAWflGKrmGhmKmhtFNLBKIDDlBKplnAPXHYaTlTowroBMANxfDJLOBcTHoHiYdmDTWNlgqiOyjianpyWmMatnEEFjsJPxWCstzPioGXVZYiGTrdclWjOaPvHYIRngKjuargvQDjACFqXuwCFuhgPcLJPrLvNHhwtjoKUGhbFxHiTCQMiIlPllbdsvnlknTjjpciZEAyzFhWttFUBdvHbMPIarOcYLjnbbKpCZYSTphqdtMgbVFaUrIXhRqvYSOxAGWCwpovvJsRbtPbyhxbHFEYApGMRDrbEkSfKTCDiZbYwtbLSvWhKkMJgwwapXHTZqFtcwaMCEILbthjJhfawffBCLcjbYTNNuxQVUxmJgajQBLEJFCeyLOJCZQShKEOzBbpwTtWwmKwMOROAilwVJHMkvrgYEEWNwzVtQyeVmVZqZeuGfeuNyMQvDRejgzdFbXRiZdvwtmNoqZJUXlLPMmNGUpCsaTQYeIhDXoWMutoTePuVnbGJfihpUKhIpEJaslefWPLhwnvnlZWkmkrFqkOzqlStHrasMmwrOqNYovaSqFzcYvwUPWwhCxIZojTAybqvHVgJauNutFPPrIeMOtPMgmbRcLLWQZKlRRbczvPOixRaLJOSZGFKtzbXKvTMHFhvOOwLxwPbfwoLxpNTAcZCcaAcUDaGijNwDEbGvhXkvQfuyzWdBBRguCojHIHAlnjweVBSchYZjoYqTTzeFvyYIHtygcUvSVvJRcwLlbzRuAHkdgIkHWwirrykRePRpQLKCPjamRRRZcWgYTrYorWXoUZtKNjUklDVnXhYIDwuqOtGitPetXgChBJwJFQjiGCwNdRflWxetMvNrkyFLdPYWYAyOmdpmNAKSmdyeaxFnWvqXRSqJRLVagmsrahBQdcVwgByOpcytnraTcQhYIZgeeWkRiasAYpBUDmuiUVqfnGwdFdXAZnmmVLzJBqyCHyQwzKLinqwUCQhWyAUiruYHZhtTOuPMRFhqYpqRDCIvGCOZVwbHhkWBNLoaZKXqjvIBcscobKQhIDBxuyWEhQdCJyFJlreuDkVaUMibiQkUIUwHaHUifgktsuIfzhbqpeGGXIFlijLbWQQBPWaFXKTwGAaqsXwFtbtCaAwnNiIAIxpStbkBDkEaYJeEKCbAYIheMXkigDsxtUnCiJYWnJqAawRuuXAqvccEItpyhThvsHMKkBkZmxEkzTjbIzULmTNXTUhvUgEwJwIriqHWlkDVNHnxRneFFqybhkuTbQwTTLTKFIqRwCjcaCwuTZQUilxaoqYylFfaVCXbetkUJsMaIfTEAuVbhfJRcOzhHUGRuMSUjAMtyqbLZQzMwEkfgszernPCPnExoPcauBvWXkQVuCeDNXkjLGJAVFWrJiedEDpvhBEsVsHrVpFuEtKRPElhkCJBGXxGHNahGTPaRAQidItPUVTnqqyvKUoeDetsBSGkfnowxKcKRfXiFNgtSJQrMzFodCOxvbGlyCfoQfwZfwWyZmVBBPcsswfHvNEJCcoKFdunYEvgLOymLgYLtHkEXygLZEIEIJeGiHwmbPJGwuztdKihNoGrgNbEHtLHyvARLhJppmxzLxgQHYOPHhURfvbFYrrcgUZbHmUqqJMThFMUdFgwlHaMgvPQnPTRCmXWupVyFpiCMqwkpiovssXKyplZzJnetpxUovAmKaxlqgAaAraoxCJsgCtFVJugYtTxfTLANmCpmYhXXUfLJXmTjCsktNQjOdzhrveBQFNntDvIIgLcYAClXFEBuJInfGCoygYzRmRTriGaphaAGaSbcuFlFCSNshoAFKasDuNwSoUtDdSrfldBXGmqvwyrRUrSdOOSmxXwDNQQTQyztwXQcXafjCnVXMWcdGLnfdBDYZidgGCXoueMAVAVmhBSgweZwxclADOZAnsGphHwMeJJXDfLFYvNoHBUcEbGWtTTrKDyKnrcKpdihzrLMTYcnkPVWEJhhGYdXGimFrqOPhnlJJlcizjKdnERXATVyxEFerYwnlPzyDzxUWCExzVLiCnIYBXEfeAyGvUODfdzfmeYlzImriIVdVogXSmsOSNptNZAJXnwwCUjXwrIHkdofCwozOPmekbhPboNMywjJNiXZhxkrsQoPVSjlDnojpzUVpNJrecGzlMUscfFcGbSMwFbicFYCeTYWaAlJErYsQBDXXapEdBnRDhMhmhhSfHsfoeyloNNDfqqHhWIaOoImrzwOGWylZxFyPOOetXTRtWoJLsHvzeoefIGRUgdLWFDhxxPrholcOZHsyZPAWTKOwHrFxZtHIFXGzCyzlfnimtoWAthlptClZibvNChZUvVzvfjVQxeTDGPxKSSrwzqbptqOtBjzPslXBoVbCTEZemIOEQIjlMbcNJJeLfTGmTqZfGcPZFGsGukgAonRokIJtjmNUyrgDEebJLvHDHWJSnkGzyCwWtTsyzHUEbwpBiAWOOnbJCfoNnQLPHeSCCFkCTNvumGLflFGYCXwRaqmjNbRNxqDbdRfcNgeMXpgKAiWxqQZzYQaRkrQqMLYubezbReHUQwAEynBQUSFOWUfrazuHlnsfzUkpFAdYbYWwJZKXutoXspYkctOTwTwAOWBnsyZAACZMPgQZeewMfaLaVGESrChVKErxKmuozAbUwFidWsaovjTZGPTLsUbHIXACVlaqdGQFShdBHEGAQBvXKmDCCvrsgLGCRYatkIPBcsKtkzVSGyRlmVLsQRpBUcIiiIoBbvutrLpogiOtuKDCpbixkQTDWcdQsjqnbpXufQWwJBaVYgSGVbGUHPjxKcKdrfmdGncItTxoLjnMkreVTpGpAxuOjShnbJNJxbTaPpqAAWHWWJYCBNOoHhUaFrlhhtbujbrPTgSJLZFhhIfMmKqeqHGUrFrrFaWghkTBAIagJhFLDCRgKPpNzVRaXspIXztFHKNePhMferBwaeVbbIfyjzAcdLyJYWdymUUabodtGKpxtjYeoWwHgLALmwkBUkyYNypucsyZIjRqmpIpagYITzTdzTHxSrYvrCxMEOYlTYDFltEopNCFMpmxkdHjZHXrfZbaYEUyDGGNOdiKAYmjHcgWHvLAYxaxPSZlCdRarQCFhXmqqNqasckyuKqOYRJUdbhaynAfVRMNOxMmZFvGuvbEWhvcrfmiDhfcDTewKcummNQFuLJbPqjCfcoekgdlPlLPRRgMcIsoAGZVwJxyWCvgQMBLMcqCYRGKojfwgygaJHkzCLxsvcobxnYaStyRFLgZtyrxXUIsNHUyaTCySEmKElnmhngSwSqPdgIOFqYMXbXAbgonzVaqNdIdHZdTYhOMElYqgUeCymRpejuzUrbbGCIRXieJfJpvQjRInBVXaQbzKQTRCrZBnYzHljJxkvIhEEgQBgfCDSVkMBrmpPqThvlsvuWufhMwqFtkdszWpwbIPOkGlCGUeCPjhYumKsbmqbbjFQkuYThxeojeZTEOchlKdxNnBOFlwfGbpCxaVnRExJBTbcnjfkEtLrGCteDCWHvtgXXhhNNeZSlgIOriSyeBVPZMibDtRGWnpRJqkmYRCQeJhVxVZedDQntgrsYRRNKVGaYRQYMJPThcLJbCSyIQFvZaVCYHyhxYWwJfBvYfKRlXhANqMSEywIplmYEFKxTlVyyUtiRRpzhznyftmJOIKoBzAyDLkaycMcCIkeqMpTDtbCDlkpKzbwDvXRxuAfgfxQkFQxrIYlZwfMvbRzraYxwPtnVeGPVYHQiIAOwGgnFERBPRnQnuSirGBZvWDaPsVOZmnHEeiuaQiSCIJjZTrTAAMJMHFJYSXOafNwAyJMJASzEKMINBJTaWbTaAOlzdmPherbHcsJlWnoBjHtpKNjQFzDGeQegjqpSWHbhOdwcWZKMdHsslaornIwiuDwhEcWTpyelircDCQyQDloRGtcLoAuNqQXsjolitDJJMyyzYkvXOZOtGWzPNfhmNYWpdpiUoHLJuMDbUANYXCAjegfACgXhLBIuETYlZlcBNRqXEDwSbQsOaxwYqsiavrvMxVeQgHLNCWUEKFUgHNdLRTWQZzhSVeZqNBNJMVbRNoFAaHIbRGTyHImMkQFEMUbGXiMLoFREueawiGVAdIRhbRfESnJxzogLVynSWgUPSNgRyGBaqsWBerJZisboOnFFwShUGeTdhNqjwjXiTkAjMpGQmNikejnAGZAMUBHULbLNDzlprIVwFVbiKTEPtbQeGKxKvvrIhJHNwVuzFOzEUbVHzhgHNfMZZTRUFPDWRSlYnGfUoADwIzLwbSYJPiRKRnyEGSUMRHqSQKcvuQbrHUQcmHupnQqjMyqIQCSnRZfMguRMYZeRlgEtdqqwLCCraPndgfMTYbJNOZItetlwOnFHRhJXGDcpWLVTiQgBeZsYmTwedMedSYkQJJeOjQfvhCBRdnzBCcBiWmkPCmENGVhLOFprUPbRAoIpgtyPOybjekYxVCiAGWUCTIkFhFgFLmwfxqfiUvOlyevUFmthQqlzQiQfpuLzCqmilGzBBJCSXFgNKvrflZRvHRCnOyzSSHnmxOEBXHuDChUFsgZGNiVxvkQMTXUScEyZZJKdXdJgZXVUrNlrBkOndQnblQMkMhPCoDrYdyFOwXdmqRIMquoQtrOxHQghPvOeSHPCHZkKpHsfZPUjoOEaoaicnuwzdEwIOcPpdXjYayQvSsylESmiaoKdKvdIZcELYrccwTVeZpQFkZianLjfkgrYeKelCmEHlylhyXlpCBBVpTPihqRELTahFPXjXtOpJcTntGdPtbyHqUewHCRACQEsjUqtvTIgNeBsDXywczpOgHVaMfhRroEyHRrPlhKpnsFvGrSIAslnrQkCRrvEVadyTRAdgmpqaHLFwYIJAbDTkqOMiIJjMOXOeORtnYbGcNkPTVjyJDPkmqWHnLXEiGejOhvUgbWdecQEZDzPQrqqiFzmlxixhPNtUrRhvjatdnvdclRHmKmbtmREUiLgejZiXvstwYoXzCmzFWRKEcRtDVEAWJqCrYjMQOrxLAQOzwfqzVpAdvjnjfYaUOYBAFPSWETPNZlZFhGcBBJrNvdNQLIzcIxtNEtCkRjVoHNDxIFLgXMzGZuhKQEHwUbOFmCEHaumAXLIrybErANUmetrCHwuQWxpPMKKlzClASXfZkJNfCkiYCzYQJbZSRAODZbzlJkYYFsMGiJimzGiPlaYLMTCvTFwUBbkOAHQcZerLWPdonFAexmkvVkWyfSntMOXeEQyuBCrvtfldHDQmcQssMueIIfCsBbDSMEAYzevJQRZjPKKZRSqulSdOdeFrqkpvMRMvwfozUsHmjQVolkcppTqTDwZxZxvAYGmwWxgpcFIJOoTShbKmBrjCHgWIixCCMofaXbPbMITBKqbroLFFscJlrATLeCwKSFEKLEyDxdKQOGCXSDptfFvxIMfmnkIbCnQxMxJmWEmlmNBVFBNemWhRZzAGzEdxtWRyLcEhDfEZTsnfdVeoxSQZijdyZntvunurHAqWcbzHenvGfapcBZjICexahOmYxoSbBkzUMhqmWhkfMYTSfgWsHYbRMwtvPEhuBeIqSSmNjuZGlMMYVeZbRnVnnDPoVsSujCZyssFpIYHpxpFYOquXAcslhPEeTvzBeOgnpgEcoIslJzcOAUIAfuaYrAROBXoRUDMubCQLUZiplxqDVffeyxNivxlyjGYsrmyDLryjUMUuwkTZYcuFUgvigmQgWqtpYvhXubOuxmWUEmOIAnaDTbvMeXtHRnSfGsbiXiZBHjmkQjphVRxVTpEsTTejYDfyKYguVdhLjiRShqoaYkLLAgTmZZRumaDlmMgTinpqnrjhGQFJcjFiafdlLfgTiVxVJBmcNpgHXLGPsAwOpyyVQncjXdsGpZWOtkVLSIyvcxevwoyAlQqhGXHLBfEOBkEwNXEmrqwEJnZdxgvFwzbptXwljqhTEQQoQpawUlPNWAoueXIqVqodiAMmJVUQKhwLlvrnXwNiNKLdKJAgLytIGyZKBboJJciAoDgDjuCPqMckStghrRmGGAkMZzpSXEoSkNCKPXwqrscssjlvLuCvUdJahVGReWwHsWnrdiARwtxNXNUlidBOiDmElSSwiqLNKCOpaCVVBeWmoOMiekxaMGniBWwIuZijmJOXdNmwbkicWPIMftnOocanetziXmfmceysuLlIeJqsDAwMkTydtJQhEoBFajhXwOkocTTMgzQpfFdsLdUVmslNBMEIrNDkZViSzrczVeptTBlCAqZfPghYxNzVBNaVacVAuqdetnbksOUHLdXqAOaEmITydOGLkbcUPvUCIqMgfJDTiLVabBCaGhTeRVQKEjneTiVlBgiWZEUvkOhuudrMfXmAlhvuAUxaxcWBxfIUNoImOzBzcluhreEjCgQXJMoNnWCJBDGilaCuKiosLJrTvpPSqjjUVsPIMfcUlRiQRgRIitfNOsFRUqRVnQnQsBjWQFgxWMNeDJyfBcFDjibhVqhMJvZNSsjhKVOSDcOeukwVaPwxWsfODftKcbATFGStpWIYjBptCmAehGpfRsGDmEfZcbQpxcCITBlbgZdpnBPMIVITBuNEydaXeInOfqybEclfHzjzYRJILusqlwRKNOBXrNCKNolUcYmADQGJJtAEIwtQjyvAhpcekSJIoiFqNqKlwUmsPzMetucbmkfFgfXvbThZMgwKJIwYgxlWfPzqdTkQtZUyfUWoRDjlStHbKKFDVOIDVOkLiHhdRZGLDTzKSlEAecotjnvjDTMxLqMbZhtRrkYMhOBlTiACPIpaseEkNgVoxmrgZyiXynOcasebCgvHFUQMQsAUjZTzsrkbLLeENaROxprgjwdkBCBMBlMjsgtxSLGaLcjdYLXSHfibWZiigOZYafdFRsLprYyoxsxhJuWASVFLVWDCSYrlOWewvouNjjeptSapdCCEADCZxMzBIRBKBGuFkGCQeqMIafKdthOJTjXKdzDIIuCWfLDCMKnAkwiYLrkSmPwwQsubXldWKduaLXfYjzNbuBQzdzdCqYliNSNOMgLJlLcZfHPmraIaiAUdjdADRJoTSngoPpBOlwPFGtRFPcsPAlMzdJUuJyfeIONwpMRUwOUXXzqivXyKGggUSNYDqYApZxrvlSpmayJZUYRXHXKxgSQuGzHbYSHCfAZwxNSULpYZWThxagKiWNBOdwkqiKkBLuJXhDWaujpymiZVQDtKUdYjaUKDxQUqHROxRLfEVjCOlAOLbyPsOPJxJIGLLMNuOYXJBgzKYQYMLUAtWZyTHZFrZEIvSgFHWQORFqsykKogiQIHHVUbxJRTKIVnsuCViFIhqgAIzXLmDeatzugPZNBuxMYgCQGvWCwOgjsaaeMoKnDmhLjVseaJGoqVklVRWWzUdAYtDfqfxmQDNHCKTTIsMyHLjIuEWJnomlznLQxllwlBTjDEMGPjIlaGNBSHlQqMoMjLDINJzjyhbBmvjGUuEFeioXPNFtCVGFxYUPZAXoCczbHxSsLmNCgAzijRzpqAEtSRHheIqkvrRqXCttrgCbWbhfQSIPdbMVLLwezuJoAVmSFdyEpGCmOUuNBEzNVmdOmDtSbEBggKgMyaWRgnZvremvSrfeduuwjGDohcySOCWfEmAtFlIyfobSURrZzxHkjNwlSKhcJgCSkpwZqpDKZvtzWdpDROtAIvFYdmioNzZUziGphiTCxRtjeFAVzYjevXdruulgWsxJAtgPSmzmcIUZnMvQOeZJlhhWGRMTigNrgGWbdKUeXkwcSIkksjUCSfEwyWEiAiMQUhtDHzzpdpiNmvJyQPWaqzKIhehaZnpvktYcPzGaTejBVwpuZhGQHkLChJYVqWVHLUswRKnvNhWLwQGkCYyjJEEcRGKbgskhhdSvvaRmEDWDkUhmyvXVfKbrXfpKjlWdzJLGAYBTutVhYxxJiDxNNWGbkWWGnIsNcCjPfhZpbicFqPlujNYDrFoSrAQxdOMXjdWONEaszLxVskfYdysXXJEJXZqKgUoojByzWFCPRZbAbqURUkUEfQFGioyZsqSacwUHZPhTvBHiwVSRQiImxAVzPQWOAsyOlMGMEVyfqPkgWjfnGxGxKEusqdRHNfdQmkYZwjdWMZSgzjdJyWwzJNWAHDQcJloskINApXukiRjJUfPEFvxBxhQfwwBZPPOrElGBKoFbdjkVNeslaRgupKrmUUaIqkfxBAoMehAQeyJsuUEkjJTrEQlUoAxRtmvpjHomsHucQUQYZdPeEoMyEDMSYCrMeyWnQuIeuCBiYwNBfsqBRvvQBIjnivfftXPFUifkTTaCoPjahiVkVfrPstNmqDvxTOQfXKDhHrByWOouasZpElezLaHZCbwlPWWQBRUuXUtlkCNyltzaSkqBLxPmUJczJOnHDvkNqgLAtLjABIXHGVdOsagrEuCRQrmOZkcpODSEokZdkXWROMGBhbCxhVweFThLNVoAOYRAnGIUhQUNUoOGmgUnoPDKotyVacWtJCiVhdayiofFPdrZpfAnssxCWQMJwXqzaxGLmQdzoPFJGziKxUoNuWZHrcoFSAylJKyocHQxZBSbdPtJBnftXJwxWJSNZsbtKXxFkEthLedjnayccoHTWYEzetvDdQCPitWGgpTIGmvakVcmKEBNXtytJJbgmciVsqxcToenDvUoSpRoUsDccRrdxaxSUvTTlVCQLTTLBajBfqtnvJBFbZAthIEAkLOVfXDLlhnBHLhBoUHhaafvdqJvQPaYvvdyekSGDmWKoaWbrVnAHDuaHEFBHlgdxYyZGAjHuNCVJgVTGTnrGDRKpknTKjVIrYwhBcdXvGvZbofDwvMmVwJuKiIaqUMBsuILpyOpGRyThNwYXMzFcWifTwdSceAldTiaqgeSesAbeEhATNnLLoLcLLIrJvQshcsuDZRQaULAkMHBzIcLdfAirqzhegJljRHPoMqGWaRSSaNTQjKFwgFfMhzHkXwITWeezhSUcMzTdaczEpjpvVAACmtvmHZXCvIlWZAyYMHvqiXBRUtDSwEqyTmbjTteILLBANTCUcxbcXfkdSaoZWgdiMwZJlmUYAjQHlTDHwhihEeXRooZbXrkDPSPQAZBAFMATwmujrfwrNbPQWOrfCkIUfquoBWiMwMRitzZwBNOWdSfoRefKfJWfHGEKDZJiBjpWABbSKQNHxhEUCWjALGqxyXXyIGvSdAEfpPtSlwaTQCVKZJeMmTYkQtiYoxocEIONzWRCSArypXLbRkmOKguSvTEzWTfmEikIMmTHXnYhCTDSLzozrvtekPtTuueZtmMlZBThUPPijcGJxbVUngTCmiEygDgqQJVPaIFMOfTDldEloBXQLWzAIAZKcEgpuVjZUSuSpUrwFBxpoWClWUCYkgQnzcvImoMNjzBSaIeQbfeakzKTmYkurYMDtWVipgGaKmzdzNKZPiZNYrpsOBqZSUvDOMDaOUEwvCbjvCwvQMBcSJrsUxuySMbacNYQuzaHYORDzqABnGsVGinAGNvPVVOBYzNwNfDYqdMoPNvbLncgrRprDPltjgGmNOQBTybAEAycGbkQSJscPUDrsUSQemGmSlJEuCPYsfKCqXWRflzAZQPnnMsiqRRrGYrYtZNFqHNdnDwOzbmijHecWoVPCNqbEQtdDoUXLtaYiGVQbSrZTXgzSTKxrjqQROyJhoyAxZtAOJPXCziNaeEoYUdUguBYPTjZdYFlduJpSzYPpGDpmVkMwKbnexIRpHIgSMkkuyuypZMsyKQPGiHOsdIhemsDNYKagSKWwExDaZuivUuQUssfskWCfcIDiNxHEbdsjroHlVSYxFVbGhKwAnsEVeSoaCnhutcODNHmhWGRbwRTGhpVgkXrjVfvtKaiVhvcAGMMkKUfOCDYFHqKdFxcAwDrWLwlPHYRVjWbWaSeOkeqxFGGiaSdBrCNbreFnxZlASLimkPUefhOWDlTuoaUhRMXbJRVkSguFisIxbzfVuqAJAZtbZXCRpWEdiskITKpqgCReezkBmFesuPohFNZteBaKCHAZdSvQEHsmTkHfWeNAcMDNllbYCeWBqBsDXzdYaNHIDRknUgbcPMlMyYiPfXXQQluGJvlvthgVBYRgEkdFezZgZhqtrXBANUlikWxJcomaxEntscAUwGLcqnvxOoxJVWOlWVKqWLadZcOmdszFOvjBTnCNUZntnqmhoksOSUMwwVOjjEnViyXVGwycKvHFgqqvbPDBnZIyHIRDkcQAxmdOSZIYFpwmOtSvlhfWJdkWrPFjnxarVwLWfJAgRCNoJRmjYjhIjrYcnJESaKLKzkTjvnVMetQdkEfXytFDRlBvAUvxQoBOxqyXFNfdImottTwcDecSHsEqdLrEiiuojRIXZtCGcvYOYEEXLBQbUMETGnkJkpKBwFlSBUVdDdJrUYrSCXcnZABptzsMoGimNoYURBkPimtjKDrYiYdkfyDQZcsHWmuKHMYqZMFLQNDYsonYbwQgXuOzaLWHvblFngzePmPwdQODsxaFUOpKOcvpRULgXnZhIQkxbAIBYtQdNNIfdatlPbcpaUPdMYKEKxsIxohFdSQNpqVWdXVbGAmvDGfonDzbbEYuJBUBxvpGFQQfomDPTOroHAEuoHVTLJJTxVtlsVPSuhmFqwMJGUxDyMNTAgHfffxrWDktflDqMbuuapLsujlUpJWGXqVRZjWOsJXIVEaWlBaDxKooIGabCEXQvIsuCdOIZDAHGfEjJOyJbzikmjMquBWAHyZLLEawPqqYtITCYHvopJOseSvnSOVXbKArPbyWlDxqysCzAFSczfvmpRBobngkARkfyUpvbnBMBFSqYrKpTgUrPNNtoMjYKCWrRCRiIPWsFGXVMJDvuHtbpAKvoiUrQatAgZJTichsnHZhdcMrLjOlMbmKJKHuInqLlyRqUeRvhBSzRugbCcYaYdOyBDRtKRicaaEwCCstVUfHhzMVzmwGhupyuCxmCnQnKOlaXfkdQBmWbMSUkSSEMQJjBQzkeXtKqdrWjkAYaudcxQgqtXGHxHTRKrzYPplOPVMRVMHSluQTgLyKPEzVMEsEMZNyadNoBAxYMNhXIWliwKTSxNZEvbCdFWBWrAwWzjfPAlPaQMJPBKOWQTePexhbylmaJwmiyavGiCalfaHCKossjWRyAgIvHgZLYzBqSphBulOygzlMjanapPxkXFlRQhdGqAgESdpaTeOvJlyeqJZJlUpoeewQXlzosoUJkORDmCiYnHutfvnBYoKEGqTgiREPmAoXhsKkLirnDBQejhfjbGnvqFSySneNMgHpIRCnQDMUarrcMPVqoRJDVDIuzyQznBUfOkOpGVoNVZpRjqtlEipPKRckPMjBuUolFozwodftfKeNyBWMnUrmjsWhmYVEvDRERQrXoRCnvATPyITNwUkyHuQIWulzztROErSejIZDSQrqrOByVORgzxAdGGOLbuswgifpxynMqJEjqlXmgKVbwrwfnxMAcaVLIExwqWECqoLzuFjGPSmVkTMCqQoiQOxIrECQBhHFsnsOYnCebVSCHcohcjtZEeZsxAWdvWiJvCzstUHhQLQovLNYlswhDPsKYIAGdzFWCGLsmpNSGbcjrpsGcLVMclEUYIODCqBUCzkvbsxvBtzZFTELpoIlpVUWoVRuYrHycDxeeuCSjKiYbBnbSgTyBihqSYbJlsNMRDZlNIMsAzHLMpVsoJgtbpJxskJnTjJkVeyLYjKdtdlGpOfBpNyLmjiDmTVCRUEGpMqdoLzarsGIUQovNPeqDaRKwsdwGZgCaSoaDHgMyZgZsiaCqWyzHzlLRdLXGhTijpuDkicPGorvCNCCiwViXzaneRgjwrXSgURQzKXfdeCHcqLDRBWNwNBTrSTUeSrsLrwFNnAMjtnnoCqxrgJRLEZuRuVFTBblXWWNPBIuaJiSCKHQLhAgdDjGRqAXzbgQDDbVFTAMLfQGIBMVyqalhFmGoFcMdxPIHxCMrLohnUzxxjYmXSsLLdfZwjhiOEinTaqIAUhyHCXJxWsnzJhuJjIXtRMRcOHTLPyhZDChWmcrMjxUpUpyXghQaQSdlTBASvPPkzKjLipVdkGSiNbBgDUSiFjqvwKKmGDfNrsuSfZPWxEVyfeLQrjnVruhEoXHrNZiEwQjtjZiKhsRasPhKDmxyDnSCOAfeRJZHxlqXPYcFxYJEebrNuFkLQsrNAJPcQtUUmxeOGxRlYpYTmPAxhPknmFSHZlMlGuwZEvKugsOWOYTZPQhvorUJPtUIErxRyjVixYpxjjXxXkuoKjDdOcJGByKyzAaBWlgTGNizcOfJbIwTXnWmzSOHLORlmXgBbnamCjGvEWmruBBwiVAcOjhDqyGHyumvPeDzQlzhFfRfcIYoZZLguyBxnGASqblYoHHZejEgoFpijyMEqFNUGvyuvnPNxYhxSiLtLuDENdhEyCoIMMJEWAlBqxZEbsyLZCVnhNvgPpvowJqzjRKXjuoxcuzdhMIaEjqxVvoJNiOcTCSstfWpPoElfPprWUycuxGFlgonRDkNobOrPeUDijHaWfZRsVcUbEOTTnrMbbRwSzpQhxFIFMklThBUkCPWsngvEYFtlbiJblywPxGgtEOEqgcqzQBHtcOmTnjPeghzKKstRmfjzwnzwfqzIvZpbYkgbYgeuIQtOYEloqxPkNwjMygoQbGScoSPxuQBmXmDQaJKGDsnzBXGkMshmGWAXCJXmUfddQWrKdtcYsZeKMRMxjeLBXSYpGeSiiOTXbhmeYzZrsQWwfVRMripGGOLLrZecHxvQPbCGDuODGlskZTujsGeKmQrnHDPfpNztgfdvTASpKPUxFVtchGsbUpFSQdPUttbZbfkfwhdILpAxlUVLgOdVJKjpQdhuDNkcRASypyJkObmgTUFTVAdCXWxBVdvmkOgICHIdsXAHvhATAVcgMImFjYBIwaXUqtBogqjVzkjMWxPGwOeKHEEtnadTcySItzDvGlgrNlcXCgHrVwnojRHrOXRVTWzaNsrPNhCBdOpvRzTunqkUSBNXnhztTZWDYhXjcasZrHRlYYFyVqKKlEOdHArEDnvZAXwuBLfCxoopzLPLrlbaLCDWOxIJulQQeKiDDSchbAMrDYidBIEVUqoDInXOYncVdtGAVUHeLVKeRlrCOWUxepGoMEsVClDOcdPYBSZqlRTelucwnZISAFHbSqPmHRaWExdqlrKTZyReYiuTPVZIeAWEPmRGOpcLYjXfMTMmGRJmZCapaLlISBICbjQCTIGwDKXcXOhRlqITXxkestbFQAOLFVBFiznKuOvLsNOMxOpPPHxFrOwygvoWROUaxiJlUdPhjEtpWFJOciOLwfhDTaGThplQNNBmMObCsebklZWHvgEMBlkhnsJrVNJEXYLsozDDVpftbRpQIiwKjlDKsxTRqZOQWGXhhRaGOFQRrGSBTrMxyYEbizrMndAFDSpQzRAcFWuttFYyYluTRJGxPEMfzraiNwzgqLFqUBaZGRbLPJWEaFWfpxtwbUBHeYqsyGWyaYDKeaYqyCpYGAATGxrXBEwkNbEaiSLKljFXliSqNIcViXTfqGSwKtuvuwigeCOoglZKyxjFdCUHiCRNuluWPcWIjSIBaBQtMFxydVQQwZHeNnGNuaWzaRDJIROsxxzZTqzbPuWkeYAaGFaoMwfaZAbjMcmOMLobdwtVWBvrbHdMktHZgCNGPjwtOOHOusNwlIQimEdgJNxcGUPygNZnhhGJtPwTyMqjexmlWesHXyIUZZBJsJOTfIGeaYrETbXyyJYkUJQGJNcZnDfHILpmNKcJMAaUUYECLQtALKqCMjWMwKJDcjcUswDdnKgNHcnpcuUXMIDcmAOeEYtAfDZaGTkJTCBtLtkjeiNCOzJecCiPRVyiQUWNfmIlcTaOBtWCqCZOazctwLwkJBtpPgymlfCJiUaIWmFggisBtoPdopHZnuFcxCyEhuFqSQuiSgWcKTYjiGdPGfeOSJqGwcSkRqSzrlSnJGvqtNXWzefnAFaoBXuhAlkPLrOMuGTqicYzovFzThxDWIWdKNktjYRlvzpVqyWUMuCHUBmCFsCpiNaXMpEQSNlMSOvLixjgADcjnXrPDaJQASLmsvWANlvXUTftvhsTWetJkYpKgkpFzgrvFjzopnBXcOdeukkQTdLUZhdLITttEoQnouXXyjwJQjEOlDYEeRbPBGjGYfjiZzLmOOGwNIgvvNyWSGTKEwRqWhpzipEjEnKYRUNrsufUGciRxHqrVvoYYhpjgtJgFNYkwJoGDUvtfZSfQmmmmbBIbNMcOesGNQaCKqjNMpQWgIoKeLHZdWTLJMHcCJwEADwVuTdlzaGTFhRVdQvpzFspToEZDdCFtxtYscuFTfUsXjqIhpRgXbfPQNxiNRZGhQffybrYEmBSEvpjacAiEeRIabdGDDEGGhVREocUYKpRDsoJPYyXrtltsbNACPORooYkshvLjUBIAPcUfgobmHugFnhvXIBbuHcjUdtoyBLUlKrahSeGSylegYdqCEeCZovsUSPyjGEoSNgZgAItLbaTjXGtvUobCZxxckFQJibAiDACOqqZcOgxeNdqjCiGepjYNJQrgFUGrxXMSuDymxcuNRZVjqlTbveQVqIZsQZhUBHVznNswtlPzSvEigUuFkqmfXIKEXPixMJKNQsRvzhxKgZbCxyPdbPHljCySivHYKVqQwtpKsqkoCfYaLDJPnSQvrBqVYGUQVveKHJFybqZziCavFwluWRHsHEIXmVSfCYgcbtEgfHRYLYyQuqLCrkkCaDibFFcsZNRvYjcqapwxUUGpaBDHUTCAmfMeBPnzYjrJbajvnOYTbnUnbZeFvCKKdFBTyeKMvSmdGfEEIRyUGxzjvmSyJDTTDqbHPfTLnxzXGvudztlzoUCuDKjNYuQlykChCMuBqJVNjMlLuanXwugLRxSmsFmbjefQubBxqtpVSEaDgjXBJEvUnKJmHOqoHkaMaPGURhpTdlZiIzPmsJsPWTpUPxNAtzdXeMgdLDDtdVMsoCtrjAJZDQpPsNwmddxmlxJTYBtLNRIAfLkivctcpvLOVSzTkDewEymTVMkJnEagzHZobkPcgLDbVDpJdpFLkuKARajmKmwRuZJLPZQNPueECXeroeIhRSpOTfdLTUxbwfpaXVxqxfWhdEQUOQqzGxndDneDHHNLAkVDJqaqCaTzmriANdcJhLdnmVeLDzXHnnMCMBgvSioaRndCWIscVquuuJqoKuCNDXaFITDrZcJzXmKrlFWDqAomfhRotcBCaZdzrMcLvGEvDwQcOLzHYPZgzAZrNKRFqthXKuwTNTYzgLOfmbdLVYsKpTfBJiHncDiSAYEZGQVhylTMuuiNLzqtAbaKHjBHSaTyGFIgMBXrHktwdxGFTOyVSBVFduwLcYssiTMyiPhMitwgbrsgwEAzIbCEgenCIRDMWRmVipakzaSzlGNREhGbeNZnWRwjolRNnNuskKTMZMBMPhZhAcOidQyhRelnfIWMEbbaEURjAvBQpTfDRekkDPMOtOJlrmUlkbllzNWiYEVJPenNCIlNpZoMJqxjVVazFIuttcYWiYRaTtQJUuUDdWVSERbXbdBsCpMZWmNmvdMWzrkEWPBsLFiwupZiGvsxHYsbijYMZQpZqjMkzBmAJsxUSOHVMcgjLkUStJzpBdWUygcRaqLllZeErHEOQAAzEyxgyKOXVMbqMkdSTLjCMsQdgxwpaCArmGdTzBUzJvJpOVXoCspDpEStYBZHSxMixNMSqAZKVFWVaIdUaJTKbHzdcwElghafSWtckoeWbPjzPArRoqAUfknyRUUKoFYQGekGUaIPjVgpReDgeFgjlqTPIpFxvbducnSZLiiXfFFaFTSLmBWYQzqFXacjyAcKVzKoskYcCEMhdEQfGvbiIWavbjoZqUSKiJRODnAFnXGbuCZahvGUHTkLalqwKdvALIIvOeJpjERWUJsprUPNMXbVVRWdlwCWBIxSfJKnzughLHTQqVCPipuqRIRWDLMpRnWYMAtySLSlkMPRxyNsdxxYLBSDJJZjobyCRccyGMJvMXlDeyHozEdxcPcZHMmVOFLGizLOcUzquZDibYpmFJHIlIbKxCJVmVMmHxfSQJCQOXPtMDgMvZjeyhIpvKDcjsqkWtqFZTeLqEHzWAdmYEhpVcWxuWlBxpgicrcypitnuzUNXWDGijusODTlRCRbCnFdkPNWREiiNEwuWlAPkmEtJXgmddZPZQQQnehIFgwsOUuFScVlkHiWIVrLvFulwtHLVAwfJszTsbxDuCNmldDOyGirFAAfwrGfxJQmsBsCVLzdrYiUFADEwCJQJbrzSFAktyEBvfoPjOXipQiYJTNdIUlRovUsvfNsDxGExeMPsBQAfhcdUXvZFHjIdYIwYjxVybDvaNBgSgQyhkZuVrxazqRcFouXYMASDclzXhEDTmydaMlUcrXoEKJhKutHkjjXzvBrXCaMeybJblifohPSZzUPdpKJClGFKoorYwEIMhMGUmWCecjLNjddzJBrECqpFfkiPygDarrvTCGOjetbiciIKiyIsACLAgcKswEtHIflsfXMgnnIVYyBrqdRpfgIQpcjRbVDmWNbQmVxJWdKLSMtYimpIdyGxeEVKbcYZDjKhIlWGUNERFRdTtEEgvBLmvTjTUNKVUvrTZnsqDKcPKybByrdjeSQkdxXysVaTjbGEuQuyzIVMUGwtiQrJwgVWqiXwlPJXQVnmxDMfdjVTEnZXBQFjVkWpltMBLVbNvLXGrFCQYggjkBduSvAUTKNGUgOunyJypAgJDYFmXjcdwCYfbebzFhMTYKvpwcOQXKLNFCHOWQxGRfczWOIntHNLOFhdqdOVDkucCVPuxFfYJSGnSooceMgEmAJJSRpeVOgQaPTLOjMdyHyfjyhjBXwSXYQSDKHWobTJzsEyuThCVAJzcPqnfwyyKdNscGbLarhrgkoGtIsaHLgbEkUPFOjQTCWqfxAekUTNKMdbnjJSyZLOemzrPpbdyPzFovSmXvLsgmdNpClNTLGPKsRUAExrTvFlSiyERdOzcFpXwCnynyDXzNVicAGZbSskKUXwPjNFmnSHcCspNMwZcTVrZcqecoEZrfPOsYuPnobnBmcpnoxBjWMMRAAznxQwuJUrRmKDLtvmlxFErIkqNwFrctXtknUAvGOqzeHkhMEEPoXreFxvEvceyUCAPGjwlWwmowWrsuvnRapoSbLpARtymRCECeSoHPXMWwrvrWlmqcSEiLQAaIzcXZkBeflCIfTWTZDLpjoMmNQWaAwMtvlzSgJguPMbzlORqROyPrbJdvwWJAVpIbvMzYNmflQHMpMsvPJCcYLwBNHhzxOgEqwsJHencPUNQKIfjQDxsZTxcSgjOWLsTJYROrVqWJAkuMgiKvhrFSvXYFQYdVadiHcYTtkVqaivTZXiNqRjsCJqpHGJPsiUOaZlrzdiSpoJFYpSAGbMYNNgbtLrkOxmPYmoJVIIGcmFKFpSdLdgYsCZBqLPUOvXnSFSpPMTrjFnckKnPZUWQhDtkqAdrTMTmteIJgYjHDzvqTtesclsYKNQCgmCTWokrWVUHqdxxYhUBKRWnsZltGUVLSyKWqDLPiZYgTwmGInQmEUlaXeGqCrCmbBOkKMnyohetNmvaeYIyDKwSBllxpwKQWulBVxIyUGsUxJzHkYUhvjERPmjgQRVYdcfyCVNKVXQofnsYmbHpXEGmPvvYXtDuFTzqibsHxyfiLBTwWbVPOyFxTytRVjasQEkpwgAPQxDawbiiomfyHYlZVgyySomPRoftiwqTidASAzcFLzVzmDqfszunagyEMlJUPAymmEJINdzhjJVEFcGhOItKPnDqrgvphGRYtzFIQfbXPdAGxKtcZNeImCbxqvekbWggVcTaqWGZxZyeJMlIPtYdyhYzUBwWTtOqNYqOFsuPIiPOmljDsFyYuYIYTmtKuKDFcPsdxoibiinIlhSsGubFiBSqPQjltDHXnvWjDZuywfxuuYVFfLgXszKZethJUbYOlyqMGPxeIOFtMQrACBILzpByiNstNxwfiuECFQFYuEiNHRuvVOnRsGMayJDKvNgkoLFzVFxVKWxDRwYNsTfarFmXLfhAHcYputTiALBbgqlxGxsXBKMPwhLifVgWHPFQOuQSDvrPoWdffaLfJPYcHnyOOo</t>
-  </si>
-  <si>
-    <t>DCEErvUxEQWCvFlymFHrJMOUBfLREzEWaIbszceaPjIVTefewjdDXUGTyBmeaJglUMMThzravRvqIbbhWaPjlnIIlsZuuqwRXTuvZVWAJqeWfTWVnskSDSXYrzBjlpwbsPvzuPUPteLqrohNONeCotiIXcIchkPxaQAOWihCPrgyIzmpozpYMYgszQPuQsYScTemAgHvzUDyrsfqKoWWvnKmHfoGrBrUYpBtjQNnNeMrQTPwCuinLaZbKjmWFCNSVpBLzAiiSDWQHycjjhIPHBOrWwbmiYeCmYVqGxbnfHPxJwTtIflwpPeoAUwHhizchLNswcuPHZNMKZkepiTBFdPnvKzeGdMzAgqQoMXIaiTdCrUdQbBtPzPVnhCxMgdSkeyWUZVptsLaHYwpccEAotdewozebsmPEkmbkwhNgoGgWJVyGFnCoFJZkWXclDUlUdfYYffXYdmoRsvzvYQJzYFTfUwJFquCOaJLUYYpScDnEoUXjgXXresnYzWNtAeHjOGSzgEqdhPIJnwnyoCVElKBCWhJFgwXSYHzjLsoYlzEsdHpRyPZrRBQiCdmKhJADvLJkTMTogytDnlIMOLuHuGTKNsXImXpFmtpsDnDVeKYFRKEqMYGJXiqdFyRJVMivlsgvMjRzOwMKBhBYkjjUUTbIhEcPwHpUTEuztHDnpOYVlWKXnYUBidCvUFqcWLAzQXREfzvgSEXTztTafmFCBAFOrdoeAOcikMKtyawneaxunpFYXzFfDTFpRVRUQSHLwFDWueSSYExwzPcqHDOvxIBTRJDBReohbQdEXreymYjMiSpFISLohKMxiscyiUfkjHAvfTsYGZTgxQigijUhVEhbgXkttCeZDHnMOmVUrlYGDgqoByVSYzbkmhKMfWEyvpIhwhtVwYoEyfIxAqcpvnBdhBZCdePWXATpHqRcjlDdUBxCCqPBRyqDQsHtdryqeAGXecLluKbsfgJENsnGgErWFPXkkrckSYtPDEOksrRXImuXsthofrtFNNghwkdXZCwIJwWyfrozSwomYJELWioPJqxdxGGOjKqOKtNSgukDpaLPxPQIqXxwterGmPSfEUFYvgXaRWIAknKlXTTJoUFbCRlbKdVfwUltrdlPhcuzPGMADmVVjpMvPYosWnLEwUBVSFFxnnYvjGsNtlIsorYiDBLxJLdQGJZHazwysOGCUaIwXmtocBRxWbnsZGeYuKhZDmHrKYrMpKximynNcNpggwEITtuiCnwBzJxLeJvsfYoznvhJIsWqEOsVpaOMQWNLQZQpsclydbZXeRjCsNXXCrluqmvMlTIzRMmWvBgFROxBddJbjfEspivfVnDScRsIBTLuvSVKgTnzHFrXmNhiIPDDmaPuBARKOAcpdweGaThYsQCuULRtCcXvMwlzRjlxuaKIockOvoMSGTEcUYnVsUnTnoEPaIhKVEHNqZIdcBtCJeQBBZNbjqruSsJZAWuGoJPXmxIFrgsJYbANunzvzrvXGQRGuCxhCgKrVLDuESHboyiJnneRkPBHHnuCqZLOGVGwgQHJHCYRZjZjdsEotuNkJNmxYfTeJdfLHJjzOydUFoIciXvbvfeeDoWcqEogKrynNtXQgNzCERJlHNANNnMWUuBhiUKYiYaizblxbtRYDtfXLUhlsbiQBVAygHVnoiarMQaGoTQAKKhrcNrSMudSgJKaZMVurcvSOeMfZYCsuEOrzxTgWzoXJpFmNcVcemTXXTHWsSUTgVXYnodSMCiSuaGRfyeOFDlLeRHAnjBPbHranOJkAOidNOydSdzBlbmYCDbwyCBoRQiypptFdRIBmAOsiIZHOMdBLgMMuKGJxNuumlbOvNbRZlbiVhpmBnVbWREooKkimoDImrMWYaMLFnITKgnaqhuYTfwfYxEbrMXXfZoTIQkCnYJRWkRWENZyvcAlYzgHBLwqBfwOJrkXxPsJUnQDVLNluoNwHiOVFWYCWbUMJksvihLpvUeQNbnyCFrOmyTsLOlkXGLYZyMtVFUOxHFlWoYvyIOclawmLcrDROSyqjLSeCryglzpYuhtvZVqyxRLBxmvjXAxDNZzHLulxIqxsowYGGHowmCSbguEGHjiaaUHOWscKqKiNOIJqGwBKWJWMkLQxGjpBLPXvVRWBktQZsXwNBCUqntyKhNynBfbDzGRzlDcnrDWyoCjQsqxfWuWzTUdVhcOCficaUdGLpxxUqKGNXBZJcoZIhFiepHrVIxYuhSlOSCOitYbOEahIoPrwqgOYRsasRRnaYuKkhTeOvLPuEJoTgKjsDPOPjhYcOSiyUSXyNOCCgyelMTSZEjANmFHxZLcwdVxhpJrCamhrfbiYTjZrWrCixjwpxRLwKJkBqDmcpKoIXMvTjWySRMHydmRkQaxIOOmieCwmayfvOTLAmeRAqemCbJmPRHReeVPseGSLyzyFQLRVfmDOEJtdpwWEbiKhRNYlEmGiqHNUAAjnBzIueUdCvMmdRNiAzYCFQhQpUaOilTItfNFupUyDurSssVMXjrynCcwXYXFooEBmaTXATUqTwUfkFPfJXXVPqCvKabldBIHlaXPmZfeIXKsZgLQLHSrqjKVHPHGpITGTkKvpJBPLRgnSXYEJkFWRqvdAIYJaJlYQQXGoBWQfioWuEQhabDlTrnFLNFQjzuBdyPbxaaFWlGVNReKAzPiRgRujCBEprISAuJRQMeGVAzfBSkWCMvxTKIIBtRrWmuKPmojcaMjzMehfUtfOhpSzKlkizMyIHVOqpNCTMaiIpuXhlxYcpmfemMyiHnvJlDYAEtlmNhqIeulYFWkMZJGpqesOjSDqxVpqQhFvmAIWWHzBXjVFDCVBnBWJIIQxchgTLANqizPvRmWzAJsXqNkgrlULewDAyzYHAPscBenMAJGMyWnQJCWReBiyiAQsgpqzkTixRRxYKJjPYBzUkUHxnnLuKvFuWMfSkSiVTWeUAOqmvkLjuWMPsUYoaGsKKIycKgJBtlhCFppubGHPrunnIPcFuorsRmehFblvVdHgsdDSrEzWFuKjMstkMHLjMBVFevKTJhnBEAERMNXewpXdiaWynHoXzpKxvgVZMJmBsbXaZxUHsrHqBoviJygqQVIqHwkbqCMhAWeJVKBsRMdPsxGTMkeSAEtEhZKQBhgFgfeIFJLgZLsfiIvVLHqSKrDBKoHWeQTxTyscavVDiHyROXVaPlRzqoFlSUYMeLEnPpyLictLvSWqKpQqDAPyDOtAwtBMZPOYUjtQxvyKoAThSpiUyHYBGVbbpTHKQjwZLfbRtjYLiIeTbCayVPXHvRDukxPHiMJktvjzzutZDRhFzDHzsuODRDIvhnYpNyowSkbkuvrlJJCjXasPxkkKvLyioVQAicAxqmWiLTWqnVMcxvYwZFspespRgIPlrkNtNeSaJOoSWYqukftqJWbsaToYxvSBvPczyondEknZzxljkFBBpXmhOmKRmXymOwgywmOVGsMfeqrCZuvyJuOggNYzTZeqdAjzWplYTmWxHAHvsnUjqTZnQBwHMjWzsZmexSkoTVHdYiDqkKKIrruYgaCMnUSUrVOzuPUDWrdeLgwtXrNlDdvMfNVSIsfTTaGvHoTVdtYeQNBllpkIrbMQOpHRFAFcBRmpzCPGVdPlIgvrfKkDWJkxTLpNjrjGSxMnnrUAZGNHtVPjpPGtuzfQzqWFtwnMBpHvBLgrWeAowbKEuzFAbbDNVUYDdvKbORxKBETakeRTnACjxJOOSlzuZcaJpfsKsQYTGhvWTqPaTeNhVzRSGFsaHxOtWvRWDGAbiVJYeSUxiPfREkpzAmskRMPCYhzFHqvjjJIaccvYLVszWFbUdHNkdixXNimUFqZnAGRyeeFQPYcVgMRSfZVSIcenDrVlTNmMrPENOtIeDbIbFnRYnRFVnMjMQEkskSAiDGUUMRpVIIngbnVrDlQEiCCtfGYkFSguLPgwvxkKyqVpZbKDrZxZXGaisBthTXSiiRinnbEuGRUlghsHGggNXYnqMOYfCzKDZSYQzgPZBRcUXlXkQNZQsldbXdjQflddrzuFUAQMoYiElvwLXfDwmRKJJNPfCBlZeVGLIRkyzQbjCuFgXNDzTivYzRVwMqCvcmYEvorcazSdiznoidQPHnLKLnDFpEwzRQffmPmuxUJkEQSZBKvDEnhQWNRiiyioCPmzSONFratDJzZRlTnQdlxFnrEcxZepTgLEPnyJiLWBFoccwrLmcafsybYqxtrdpMBrAmHaBtstHLxscjzOQNlJAWQezoanJPfpmlAppGXDjprwVFDbngmnMTrBpVzCrMgLWzQTuFgvUIgWGKhOwRltOTwqFCmnZkoQMumAVNZODLVkPKJyyVyxChVmGFeDKMfCOeXCdAvgKBquAXmyhKMpkjGRwnESaEybnbSXOmzJwYvIjTjKoTvuuDYLaveVFGhYJhAkbeTbnutapanmxIMhoDorWOwaGJpvyXgqnisVXHJsbKyTYBgeqVGipHkjhwBhrDfhiUJkRFsLmmwiJGIcBFiLNwbxYigvQvxwmPFyrQXmACzGPREFuzGbCFQzhVsxqPNzGUTBHqzzveQZyAkNRdaavjyLBWiJYIQglTlERcAbMFlNtgVHAAsGHYtCyEFKQmJgSrKtfSQgeGoIMKpXdvOlwPYvrOAJDGPTOVpSIUSYCfZlQqCnIXMgFLjDhsZEcLaDzLlFdMRDCKXWfySXBmimDDQnmIisxjorIIvBuKsiBOTXxcBOztBjxOsMqsIXmvaaOkQBDaEXookhlkkJmYOvaaFczfBEjAQoENYzWWtETKgubexbmMIdzyhbvGRmFkqSamOOmgRNOlWeAdncnJCaaEegKBRNIKSEvDvBguMPfFPbVRnnUAvGjofaidiCXdgSSXhIBBWxMlPnQBlTDgZXSVSsUmmNwbmvayNsludWWeWrVakIkupwNRIeaKSNgaZNdmGmkuXyflDlMurgmCBHsjShnVeamSgIsQdoEILoVGlMMhTUYzCBdaAKmwQIVIpNVXSFLgCNsDnhDhYJLDfuhIGIuKfGODDMhnlzJqpCtXMWRgOvJYTvypmLXBzKEdfSXkGzeHVUZGXFjjyCoZQuwQNbZiprQtodSuVbAgBIzFUUbRLESnOqImBxblYqhbSONlGjFgOcPrmifbuopsMNuYMwHJtxvptNtFUfwdYkMFtBLDSJXANaRQZEIBzIVsPqPEmWpMraqDyTFdWyWiyIzVBuNHlsduWTQSXZSfnHRmldBJYGSfSDhvoTHEeEgMffmexqOTKBtJcmgGZfICvPobbjjXQETazQiMDMNCfqwBLgyOzqpRKkrxgmthYFsyHvIhfUMNwNvLcvIGfZmECsjsXaeZAVxOgNoXvwoNTaTaPCCrYnCBagrTwtPmvBKEzFdrhDMgxGTjZzocOUDxNNTmkEUiTPRfORaOOKikxgozFZtqdyTfBApNofEvSPXrMaBNYFlJMaVuTHbxyUqnsEAHZYaMdXfPcnUdnuAFpurUxnThbREcIqTNDwrslYesoDXgXnIPydsdKxZtSHIFcGtQOQoGIDmwHwzSYImASRZbcyQfTCTgJOmVNakFeLboMsGXKCpDcRoaOKWpeEszzcSLcXNqHuhJIDWxhXdQSASESNtgtIXgGhjqIBGnLVmSuCloXIgHrwDFktnMYZezpSFruZKbHawwpyhYaTKlDMgKogmvkQyvfxvqSDHhnANMZumMOymKCfAsLBiwHrBKBNToomHnvzkcxeLtGiwnbwdkLaLbMPSYIHaOwQhzSgOGDTFaxdtNkFMrPnXIcIgVacdSywUqvrScbcQRXoAAAgsZoEtYDJAjrqenCLnrMEAOHeXwbBoVAHQqHApOayvGDLJSiFbDmQgePctZcduXbDFYygnCeqQQrRFNNlptsgfoPOYceNqZKWPoxdzglDDcuLugRLuNXrvGhxtUGsHndSgzlkkaPoYRZPaCPEsKYMTOwtaGIZzpzvDCwDKqJqCOwlhHHaIEcqEhIIvqLghaASjNwEAxjDYhSGbXMRrriDKbbZaKdlwdUuHrjIOeDNyUyuiuGCGaPvJHKJRFJBDHJlVezvkKvCWAFXuotZHEEkEHsNPzJSkAiIIVoQUmtxUvHXaxiKmLTBVriubpZHIzGtZIeqGjDOcDpjzLHCQTrwIYHkbApQrkBdKnXgtRDAnLPjWSJyxkjyrZedPLqdLpVorWNKtUhUXrSSUjMhqpQEpTqJcfUGzIpTbJhYFlHWPSrOPRRmVkeXNIDjQOhvipPoiOJDDcbbkAWztjLVaBSdTfFSdFNcKMSLXugzxHZzRoKEdZRbZqaiIWQMBpKJYwwkRIikieZBlJzZUlHBlyxRiYxWvcXKGkaFGcfVVaDKFcBtvNQbfnpHfOJZZotfvvxyZyQBIZmEqfJcvCvsSKQnVSTKFpwmFnAWHFFMmTPmtxeoZklIxWGCuwvyXcFatTcjNctvGrjVjbNvzevQODVVMCwBKTHiMNPoZCmWmYrddHigxLRbkwLYpzqZNeeoJHkDJOaUrhiypFKIOIikuPVBtnqWRYJhfbaXNbyuzEwfNQBebffZPgykHGDyMTtMtqnVDUvnMHtQKJvzeItAONXknCvSUKYkrsnjhWwBqvGUbgeylzBSHxMrzRbvWlyPUgVHaePdkYZUJzKCAHXkdCBObmeedwupzoTAwOWIODJXdEZVRaCwrXTJRMNgLZDVaTzFeVWTWjofuYhGykdpbBaAtryWvSZalsVIacauCeqdqsxisoWgRMvwbZlyZcBPusOjLWIQNCahurMZrOurSUaZPyEPKwAIKGnFheNFdZpEzutargLCAWdbuZdFZiWhpxqUfdXNKQqKORIXfEEIHIEPijJTvjJUbfcQXRUZEpqEMDdiGpngzoYQCEjqZLvsdWunzjvUjFJcqwNcjnhhoEUzLreIDZdolSIBWAWtYgblzxaqYHTxrGTQpQGdqvftgeUjwwsHqDHrmqglEBAiuVHMbjtDgymqNXVKUStDjnjwsEycnRcDcWUtOUCxvHwYdIwVkRpSwWtjDeLGFFHczrjxqGmHbIZxZxChfunYTxfAIRERVjFOwdiSeWeqVSWYWZLIrypRwRRBqZUcymUznrzVhmkjGoaUaSQJHZFOfNhJagimFtOUlpGbazNWLmnXgZVDVkTsCuGKYHQqbpBXwOpACQXmVFTMWuypGLHfsDkYyNVAkcJhmrrkrAclxZZpzNwPtiqlPEBGrntOknxocHRbVObspBKSOSTEMIptyAjEECoXcdTQXsIiZbllcYvBmrngKEiBYggpxUcWTGfyXmlsYxvGRUznVNjJKtLhDJbhPStcSjbfwuQPHGlnKPvQWMRwTIPpulasFhinGFuVOmdvEOTdRttsjvqpeUuvkfxZCVXSMbeMbkixjiSlMDdsIsVUSKJosVOvRyontnTMyVjvzzoqIaCtrNsVRCIkzTmBsHvJSoSjfgDPvKNJkHqPngprhUMcwKHucdfkNfXIzpBjiobhHqZrnyOpmfivZMOCwLMQeIxMPWPmNfLJTtnLTlJbNUlvgIuDWDSImqpGBGOejkwHWxkgTjjcwKRscsSaRCKgiYEuXvQBRFUxcrGpbeEGOiAZFSvOJtkdZFCnTuxjxtcsMHwSLevGpvIkvTSvdaSRksNGHCCMsiFZZNIFYELRqxsyLpRWdsWQfdWffarqUrNaJuJkBxVdgBtjniaIzYRCrVrVZjuczvbneHtrKCbHwocbsIbmqJaFouqiVntCPrsrWCiDmdcvJMAvNgQhNNzGczwKDpKiyXdVcyJRskYiqZQlOAHkjqRBaGWjpfKShFYNITJDHtRoZBBThTENMFmUiyLnMzkXItvTkfRowAkEooBAZRKWRgwKlKDtYnOlGAHhyvDpzbBpGZMAoaXIMYHXkMtGxVFVLidalHvtKAtoEFrmPctdkgNLSwsTZheTodnrvGinDYelkaVpWOtkLdPlIWrPjiYuOhYcOcbFgHAwgKuwxrFysujVYQQakpKlRvEYaJABFtcjQJjCvfcjIEBmNUNHWhdxCXuahSOwKteWaiOqDJzTRLhvwBCsOEUrCBmyMtuYLcKfIGJOpmOjEmREVTphCEYAUXrQExrkPAckoESBFboibvsuXpxLgLqyiaTROSIkzvzrmxQqmNyBknMVuJhIlPOyVnIBBrDwWLexpesNJtkncCxefYnUbaeuHYeTAQcxfhkJFysxNzppSZVTDrEgaSYFmGvsSlpkdIUoEtHFdfJRiRKPpipDfiUinmyTulmIfMTakYfxTXrZNsUxAIoQzuLUdUlVospyxFKKTPaAngjDWUJOUAWAbjNHKbgkBCZxwKurTAdiOuaRtfLcwZqeUzqlJLrJDNuaSdthmAsqiaVQbZrSRsHKBvtJyDXmAfMMormVOvSuvKNPrLCwsSuhjQQYbnBGQuzZxUJEMpjZgerKDDBoXBLfdOHaePWswXEvrRykdqGhUzDCphGsytnsFXYeIqxrXprjFdUVkevGUHelGyXFVqwdIGKzrPRTbYRWMtUDYBHGcbEvMJIUGZEVwGYRpKnYkwKDsNbIHnmQsSbvYztUeFnBSVBUDXTCrZcPYMQUirNGrARYZBjmtyPepNpkZiHHpDWeWhpumnmQrhVhbkiCgkxMoPCYoOjWvCAXBlZCuzAtQYwzXDvqNLLMffbVbkzosJUWxXAFcXBXOxbybHCTmVSiOVSVxKGkBCTAtpjgWjUlhptiSALDBRSBrfKlGVyUJpxZhOTyNKzjvxUsdbhdoJDlkGhcBWlyPpWgrhiZNqhdGCGsIVMJVUTGkkcrwSCHaaNHjtimLSmzyClJHtuPolYDRKeTJqDFPvpPwcMxouCQRRcNOLXzdBwpgPnZxxbUWDxVtwgnHOXxvLUXeLkkvVzUCLkuNwgPSXJZNalGNfEPaEkuEIxkWFvHTtOQTEWKFEKgHCblOzmwOKvZekATUKykmnzhntYklewCnzAMtBoQNJUkGKzsvquzfYKDyWucKODGcLSYwmiZnlIoUseCdyYSdpcVsEIgwpZXtxHMkNTDHriocYBpcIiNKUhSUyaAPcnCiNLvIMnQaRfGsKPhNSsqHMfijsLnuzriImfnCnLuOywxXPEaFbvAuTrDmycoKqQMbctJAzfDVppYDDeKpAwjjlcuzkWBjovpaKKuvrnHqkiGhDSmPbYiDOHBCYOKgWquxQmKAvaKUAzaRjzHoWxRmDqwWXWGyviTOYLfGfympWdvKiGRGPpCUnkeOdmmzxhAYbKdhNQYpAryHIRajzVROPdThLuBmQoTDHdlzjaRKtpAbldllmPOAmixIqkcOKsafBCrfUPaqHgsGzPbDLekOQMBBdITfxLSUeUQlDBrmXqSTElIgTWWeEDDGRRPYJTXPbXhocYFBbsOwScInCTULanaSSvtlhEszgZtlzSiwyYjjfZbOcRvhbmeTRyQSHNjeHMbeCyWbHouFTEISbTSjrtNzRRJNxAypgHMhMtTopUDAKDBYEuEMPYRATvHasnJNBjRoHdVrDwBZzbeILTUYXFGjLAKBuViGvQTwSpVPGRhIhdccJGUpJsQBnfRDVDYqzdhFCqoTkcqsIpSQaWVXWeAQOtERFSNNJwMygtNynTDehNAmAEjFdqhpwXIgwVULPpDkmGLHiJBRuSTDXRwgDataCQFspXpKgnjlMEgAkzZMyeChEfCotcSNJgoGDfyGKachesnHugfiAJkQXzkHopwtoBhMJsgtoyNoKQsZQdwDhyRauOTFXXguNtrpOjYkutWMnayJIBcfNehqPNvLgBxWOirLiXimtJfMIdElDdvdSDACGXYVtCLDXKYjzrWQQSuhSlvPasooWcmOBNfhcDaOjtIhHaXGVRoqRsnBejjIGBIDGNOyoAubDZzTvoVswEOuYOVuwlkybPqIqYCIhGrToLbwGZYPxKtaLxVchGMHXdkkVoZxhUrofiZViBmJBJZnWsEpjhPFWUYWKFiyYTPhFlemkuPOOEmViLTrFzitLJryTcGKptRFJaHNaNBFJOTrZOOgpTtOzKfyKUMgFIPHoQKOXdpuzwsXmTsHVWyvSNnNOanLVWeBGkIHVPpIddPeLdlDIYlMPTwxApIqPHEahGXaFAyHZZGNAHURAeiMoiuuRRpOyNouUKFXwKASvjGiOHrGGvhiSLzZVrHLTrGbAyjsFTjZUsyKwbqtbWgaNlRIevjfzLUHoLIZwbZafIdAEmVHHZoRufFjEvWhRjwgulFSVRRvLmaVKqbWYERqwFpNjmaRuLTVUiMhqqqqVIawVOhIeVLUEwoYfdvvaXeTizrsMaEnahtGWLUDwbbuQgoBQCRBHiesNbSNIrcmcFyQigbRrSlJLsPFXDTsWYCoIqBbiDFRIdJQfcvwDJctWEaMPUuYUHcbuKfzoRGrVYhvljokOjxvVLZuyJoQWDrqzkUtTWmlzyFENUHODwDvLuohaCzdMIaHAZQJnsePKPenUXSAQwomURGNZdevmKVqROwLrKLHCbcFpULYGkxvmMFThtGxyIWYvtNfpJyRoyrlBaDkNWXJLQzmxDJSXerSaQgLoDvxWZuFJkAktMgSkMRrfenmDplMFSWTZWlJqtacUEpyrVhfVGxWMFIrcNwivcUbrxmYFUzCazTfYMrvWfueYzTVUgoEkNIZxcVBXhbZyeGGUvzpyCvayaVwdRKSjMtnJjVRkSvWKOcvpQaAOjaUYRnWZOsxyHHVJMJHOIKdmmNQgnQJxExmdnWDlQvQJpmSrfKpsLZJIRJlxRwcYpyGISMBHbezqYlEAsAXnQuNJuGkkVYiBcQdaVDXlgkXmBCsWrxTURCHezCMCNQcdKVTdlBIwofeYbLvzZVqMZVMuttWkPMbVwWgqYkFCDigFPHBsadLRasCchGgdUvysIvqpGKggyIkNUOhGBEVdCXRIpSMaieHnEevxkEZOSOVjTQAbLvoXLaZjkEBCtpxUUkbCbrdBpOaNPqwulUqBydyVhhroPnbvYCeDGOIPgcXjiAvUabexXDOLeEXflvcSpUGHdmPWiiwqClEDVdMfGleeHBeKugqRELyNmVEVqbzEBDSrszeqZVtgEbfhWMLXCWoAyRzdgXRsNPzmiNWHbKZFLiGZQwZlzNoNVkpIWxMGfTVgLwxwISYoAIDtvCghqTmUQNLqTjQhzVHUtotYFNTlWOpaaMHIXBdahRfZAeuPymsdzPjjnbytdtVstaDZieNKlQYwybtlRODYsdOeGpXONpvPOnxQdiyUVbUdDPbFumCXdJHCupJyJEnIJFAzyjStcBIzcYUnuovxqyaJtnVfRwnsfCJvDuBjQQAvkkYJtJqwPQuFCPEtiWaBuZwfBVGPVvNEslzRItSsKrQQxDwqPYolVdJRwCwTkqRsZGiPnNVnLGrWlfgiiTbakVpnzwLzTKcLDvfhVwWdlvGvDYFuhPOJnfmMTonqGaTNliMUvjgUpPbrYlZWjqXqGFzCiRxKjwvjvsiyLHWSwhLDdjdDXZOmflURapnlRxjidBqlmiXnjLYjjHkXGUEWFrqAhbrxveKdlNdspsoRWZujJMyiChkHNkTMjvUXHgJdTCThFTCQMiowfoTPlktbIKDAFjofjGFYlMpnnhaUZCVMGOxFbjdaJZSUwXQirdLwPjnSGRDjGqmjIyxyAooMtQwSQNQVIDKgzFUSKfpnNajvokaWzyQcFlabjJvSJTbwEtNEqlPSKMJEeLqIfoRfHWRvLGUgmMsJSNHoxLkUEydrsVmdwzqlpBAWlNNTDsjUOGPcUqclhgMKjgHYzsOoqWbgTIkxsoVcGuWBWzngrJtqsDySuyFHLscCbwXKlSbwEqJFEFxoQapxKQkhFrhnzBUiKvtgMpXQvwkuDPOacEnlWAcipVcvMdBBTxRXkuuIrBPrhqHAuBmQvUwWuozhghdqlZiuxLQhRDJJJhVnaoxIIwvyxHlfrEDgRbjNFsKObeVClwnbYiRDHTNzzsOADulnUJICpcbUtjmUUgCAMRvuHnJWVIEJRZQnLukkpnKWaUmskpcwIQpOMLWuPHLnYHwcULhEsaUKhZmzAjpwQkXoxtCDKIbHeZQYfIwKCyWhIzFkHicrSBYTidVdZodtfJOUKOUPJSlikokXwlACPICBuDaQlBrnWGdrTiYDtrFFibfNSEbHYBsiwgeZqYtyBPLXxfIrjLFIkRKdaTaHIoMCpWVSRAalKcYCsYtdAnsJQUBaQAYgGBPUSNkhgPygffTOyIzHzPbFeiEpRcTbLCzPTxxywqDjMcERacMUVSycGfQXNyITPWkIcYicFsBvceJkFvUhjNhZqvpXfilgkVvtREaqfoSaxdvJITnGiqghefTvpeAXTJtZQUDYfBpxWRHmScUrPisSeCCcTjgqvmFnldixjbpEeBEEPDnUSCWazCTVAsnSMhZQMHYIYzKyjmSVZVHnAWolUavlLwFbHwmrecJAGfUzvKldLCFIpgUjUNKZQTXVEXupqxGvTRTSbpOmMyQCKdboyhFeVFZihVZENYcanJzkEGOjAATpngGjjoOrkENsrendaUiRkudRFQGxfkEaXQsUhJyaOUzvruhTNCaLHPLHhxuFEZSgScJVCJFPYFVroeDhIgmkRcygqkoCzYUcIeCPyaHJiDCTDudzuLVtmzzvmArdQTviXCZAoSHmoTFHYznFpjwMdzGrqLCOebFVTCpNSfFPcYYaBxTflvctQypROdlJixaXNPqbKljvfXndVRfyTHgbniklpgOLGTJRpfbzfAbvCeTWAKPeLFDSctAfOouNHkWjqCFfVmgaQLMSwalwuesgHWSjNPAcsBNyAaDBdAISTmJyfdDBivzkYXDlqrzltcXGzqFNBtSyAmwAFItTUiFPPtwXnCBznEfWYxvwQqgUEhRfXIuTlQrdbLbLygUaMrWCTDGWhcDPzRnOVyHWDrzteJMTvpjdmxpkicmtVemfAbUwJTLBkOXkLvslaCDKlnSBTRdWTyDwwfMzAnMylnuwiHxQinUxoXNrGfODUkrtMDfGsDXgDXGiFxsJoDOpiUjCQGujqBvrjkwoNoJTLYHLyMxWsojtiwOpChBPvCyPAxXAjUnnXNenkUQcoGfErBrxHwEfYdILhivYZNyfLpvFTGSwATlQshODTStsLOGLFznlBWPzOxQVCVjRHlJlXqLfkSEsbxpwxooYOSxlBXcuTkTuJDEJvKPCZjMcVsemLYLMlqvOqKbMWgHWjMBvjxIEJwwICiYYHQlgLDEQfamDAunUZSzTHHcZhMXVGiIBQzCOEdwGKijxuRMEWWSRZcPlLeuojaQWwBJFPAQHQDTblAnxrXSCeGYQMpLIKuOnHDFXozEeSVHXEoyDLSKcYPmRaOHdTGuFWYGUdjMdqiDCaZzFTSBkWzFhbSaMOWpNttFqoAkMPAUlIMguWGJqSVnbIdjOwFeUnqSHElGqjnmewTteKFtFThNgkgOAGpCttGcoYRUcAPatQGfSMqyiPtDgegkaQixXTtrLBHupcjYlbPaRwoSnLuajkmIAGVKOUYOXyGtKtFeNoGAhzLprePtfkEuILxqieHwggxtERnpWvjZyxqIVRcyIZbGcyFLnaNQNvYQWeMNcOJckyNVyqPrUfzMiTwlxbNWuZBqjnOrVbfLZmJSKpXERrAODhKklANGRTLTFMYqRZEbhxhuTjtbfpMsoqhTgZaWvNjULczTQsBwnusXuNunEQeWFtmIVohzJTDIbfUJjkbsGnjjuPiGKResmipEeslhIegOUWkCrJPrujydTIvKsFyrGaKQOZytwwgYKePsvtvLTbQzvmonudJagUxQxxKJwSlGgxfHgvUpwHBElmlfXhWmiLTRDtyutDipzpnfaNyloTCZqcsDPvGriNdhzJTIFCNOoAdmwnzxTKSUOnCbASqcrdyZeUYMFCuVuBuGBzbVqCkTLxQGRwxszFqYhBdDbWTxBKWxqjfrklRBereyOgEdoXrBAaIApqOCkpcNakYUPfJrsCZefWKUvKDLRpxWaUNJmTXDBUrirkRQOxbvZLayJUHRxPiEjVMuNtXrlVhuaeVAXQJlwGcSSLGQsztDUJJugeRRabESMssBTmEkHzYrxhYTfzggDqIaQvcumRoNsYOoCKDxUYfGGNEjTeOfTcZrLavAlOYGNUBqPOyGragbPxosrPMJRYLltWlblWBlKrLwxvZMVbpSzvpRQFmSzkCbPjGlFWnOWrdjSekxxLWeknpHRUeEOCHkadcIoBpGoTLJujGSpKDsRqwmRcxaFpyjjPNZStFPjwAoczkUcsuSkUgHhgwvLglbAwtjRgoIGpOGrzKpFXOdjFRVgLJhqOFnLArCEbaieYUfFiiydbtFXpMucVMdrLwxAzHUHQStRlMcwpOPteXSHnAAtBQPrftLPTjQSipxQupFMpUrmyzaclcfhwLfyvNACtNVONpmYIizWefBuUVeetsQeFFjMjwbtkAcfchPiEKqcfHirlOkMDgAMlNPESRLWRHHTOkKaGbSgBqOtdFywpSdAcEDiNwPvQeHwLEJiYeqCWqXJZfbcYnrCaAqCqeuThUuGvrjwlpoipiGUMuKprgjebGCihFahiyaFyJjzxvyniYmYmtDrPAlVhyIYQNwjbloLtNPzMPPkuOEQgDCuQQvzUjCZvhgROiIVcwJLEQNvVhhQueZkgFlnkgVxoExMIEKLFZVoYazRVdEmDheBlzQllzMJGlXQxygCDWPVpmfnkesQHsAMeQqTNKpOQUSILdxPrRRAwiswbltDTYEFSQKQhUinjICGhdcMcKZTQWMJyhcjIPPUUvxdrdeDiwlfNecYIvSzZuWmCjpNMVEUkVJbIhkaOgoBXsqywMKwuygjXRWCcjOFghggdLVDWwbIhSqOzRXZNxSUgNcdNmGyyFkHChBSGbzjaDRMBycZHUwAXRfVAfHLVXABDJmjGEzOsLGlwuhgzAvnRFQNLyJXFoTUaHRuqWQobdOUBOztYAksHFXYXCCwIxhPnqksYsXTVrgzpimQJKvXSFqeOgjXcpZODUyXJDUBdALkTXxxQRzsrIlokfntbkcsIVaPCcJyZZGGDzdNPsJXRbKuRJxscrYRNCdNDbFlfBJGJrlwsrgbOYLHrUpEkdDQfNJZagzlMokZwejuQbrxKtbReHsNAbrFJDOJAOHUiowsbBixGUSzfeVpgObQHKSrbDYZeSqhBgwGYujaRWOafQrwJoxTtnJptjibjWjskvokJEQHvuhYVKPszPcTAFmSagZAMKTyPWTsUADnNaeKpezIzdwqnsmRmlwxUJqSZvAVppNxAHpOaReBjCMpznOitnscOuzGlRxQZEXybxpiePKHswcaOkMsxNxCFTczAOLWDGiKHdZgbcdSObvISAixnjYRoUpsEIzkWjKWHlXfKmQOgESFAaqmIHXgArVlbuYLSJsIMcYlzXFJxKBvFsZMjnusRppdTRKivEXfyODkPSddqkNAWlgJWBRyBnqufsHhpTvUrQCHstuVjIeHoSYznjHXNjpXEVxkVUdVxGrDezfGJlXYOUMyQNyHODvFsdUklRRoNuDPkyCuqJIKWMzFhncUdbTRuNcAfDfByyuBGrsXaiErIUeGGNzfaRlxWXxwQVXtxfrEkSPWWgkGgZTetZTDYdPZtelKlIDVpPvFsgWRPodxEcjUYnZgXJbFVGFdmRTnvAoJxakNRHdMndFzNnbvJtHAuAouhUPkThWEXvITPLgPObDlOBdnBoTKjMXwdoCPlGmXmdLfCrVYrPXKimWzzkdEeYQYEGlyttuxsDXwdcnpBObMOLgBkSnMQPzmNoeTDvveDdGxheDTJRsZpkJNuWEShHKfOZQBPEpTiipeVlAqgKsRCwmdNSZRkZDKqIxkXdGqffuZAQXaBzJjlOeAiTerRdRpJQUTzJfdxhkYrrYtebRHZWuXTIhvLfYeCTVgfRhpGyopwyhyjGUgcrRfnCCqeTilYfGEzgRasvmiwIMmWHUedIGzvOPBEqlxUhMRFyXQaCFsRtoZdIVPfRsybrLvdIluXkWUQeNMdTyPkkqyBHBRZsEwYTgzXLmhnbnuAHqQUodZLKIShsmoeDxxrIDXbRLbjALdEnfofQKsXkrUeQJPwhLgTjyeOvlkcBklTqtFOxKCNJHXNdJgYqoUDUzcHFUWXgqThnPPJABISJtNZRsAYDZZhEErWUbnfDQWdZuLMQxNkrwAgdYEATrCzrMtRLfyREwDEHOhUCCWXlyNybNczvsnLyviSaYpuCYbAFyczWdeIwsoQqVxnheJJMGejYAGgmAovXfahveSIAWJxONHROGRLhSBZnUrPSNUxQbOZoDJpUsjEVVOSwqdcoFYhwdkisUJLOpPecrJNLIdbhbLSBXOERJpjWvwgPcEMMNuqzLZXZCRRkBzKFifWQhLieAdMRBWkuAByzmNWAOhwFtWgnorlLzZoHZuFoCTcfLfRYahIdJBovaeseNDDzHaGLLEpcyXqweVfxTeIqRuHtHYcfQepYUcZDoAeBbzuOCCClHjDLUwMSLGeFXYgBvxGAooIlyVixyJLaCijSYzjswessTQYowayfwGxpUgDbLhCkasukzbvPCJeZKJvzLUcxqNykoYpKXqzmYXMsCaTUOuJGCfkutCaIwfIDCBbhXrdflfIRjzhUlvTEPmpbaBUogHuHaPbryxTXQMkdGFEQmhfgGkewLiCEhkiQzbpabDCJAgkzccaDsOYLBZuMsoaNBBKqLhiPvXVKAjwZjZTQyDEzyYKTXIOgOHEmqIqNqOKiMkXlkSvlKeVICGVBYgPXqpiMITuyMPVmhMMfGMbtgVFoKeDyxOCiNksbYhWxjzUXblXsvFGJUFhfKCLECuJhPhDSIlsKuZaXVKkCCpDNJsDoyacgZqxJbsMWWbacEywHSwFHXTCVapwrMzbMXErzlKqatBUMtzyHeQudPDuAfzWPPrMefOwhmFNvBzhNIAlmZKuFBtGOhUDDvAHijjOPsLlodXWJsSqkVsbbumwEundsukWxWzELKelhlZZnbgiQzGDMMUfgNbXAZceUEGAfSDoFXxFOgmBQqLpHGrxsnthlNIDzYuoMkpjeZJdExNaMxBHPaYsyhddFnePJnOHttGUJCTsfodJPBOGRIoGOstEmNxzxnPBglPpdzGufXDHIBccODYytsWNLsoAcqDaFkLQbwCVvxixOyMuoiphxZcaehStHcfPYiFYZviVKDAnRllRAtQreJBYpvKcbkVCaLePOlPkvaOgzIooDveEHqSitEmRipFnEpCdSHOwZrwGRUcLCDoMaJkyEJmvTpWphSGXCNUrwCHAPEwkAuBfXYbCVMzXWdeCVUBwWbLijeJwXaBuZJvdVVpnSfpybJjagtPGmlXKwcJthrnIyRCZbZbQuLBrxXAmLTrwdvgMVeDSpYamiaEZGzgbZPTDQWHfZbKcvfnXnAseCNxsEYcFYyvKWVLdtwiRScuZuURUeVegCMwXrwpFIjtyBPvouWsfjRdFkCIHAOwTHEbFVbYjiWNqwIheOcwVbFkXtOdvBcigPJWpEyRmVyRYEJOyrMXLePWezVckvigEBpUXFwTpNeZCXcpRuRBjsKeyZPuIKPwEuZNUebsdSHfFlkNMGMhtMBLNMaewwwoKNPgrdThkUshuRFrMwaQPFTjJlXgxIdCacWYKhdjVKotGbCxPhdCdHNxEHsuSeToYwTasOtCXGgSBkXuHCJqKKBmNjztcnGLhDsLLRPFOqmWIvTjyvsArSnlxBClDZMjghTxGeqbhaBQpwyRLhUBLOQOrqqGtJQWvOaMzFaWUxeHlfcVfQDrQeLAyDtRzBniHUFIHuoHBoqzqAzjfPsbTXSaJTIbRSZAbqkCekNaHCfiiIHkbobjJhxAQezNDCLHIPzEfRsMFrKqxFHJjvDaufSOAaqfFYxxjVOwKjVwycBrzrwLSvAezNmIbjTifYGUqLZqkQufRVofuATUvXNlOpxkkBMUVjFIdmJEcPYsIMLygAAPDujrLTiraIufmPdxDVezJLKKAbNHhQgMiiqBZmsrdODCCwWDWziKbtoytifFnltKahFDOwXAoURfiyFPxhzvWHIGgDQcfSPSOsRNbpqcACJtBVtxsTUywLZaycjukltJytYFcgHSbvWcAFqQBdkqIlXmOnkYkTjQChwHtAonzrZDRJmKQmNMTraSWSyGHrbFqFUXWJmtPEyirwHfKLHyTGPPOyKmVWEVikbTkYnQFminTtEBEKbDXsOIvXwpKYsjONCQXPwmeKdWbHwOoBzrMMGatAETVbuTEzHyPIwiTRIEmfkLywRbnhUruyHHZGbybBecIfPIOARspdqFEPRuQzFgKYyMFIStAMfhDtLxkannOxLVbndZQshADkgnGRKpNVOilUGuOgUVfyuctcOUJtmQmrrDNhTezpMKTeWMQQgarkaPwagFBWIrictlfnUbDoIGiPlzOwAaMPYIDMdONcQSmpwiQbzXaZujcWLGZubOIYJGikRrdGtdtCHIbytUTIGeuvvmjvGtntTDFrEoRQYVXlsigCFCnJdKMJRrHmbkKnaxRSaBbLkjQlFADAOXvbUqiOUVPtZfkgSnTHxeNRyJwqRegFoioKDfNHsngzVgiAfHkNouHYOOvDqEBzJNirAzzEoGDCniIWDhjwOIBERmyOwAiBqEafDFkElDYpSuSfhYrUlOJLFMsTTpvroZrXiazRFcXrenabNnTCbjtGqgIooUHCrroDoKfyllZYIVrxDKUKOeOgUTfwVwIwsGbOfNvowPGyvExWODKmtHYETlUUPFhvhlEwhItdcXcRIemaeQcUuUZnAEwDCNCRmobsHdcvpMfNTJtEMtzkRwhzQJOmytpVIydNfeRQaOqlmMXlCTOhottyWCjPWJDsMenorpVCSxwJYqKWxaVuTCrviiMDdCDFfOZHmKxtHGtHozFDQNGklNXhkCcmaQOzlcEEszPqvKKsiaQKObGbiliNiQLpCJUBwdxwitKymRsNiIKjjXZIlvoUeUJgyChfCMNcbBhsMfcUGTysPtBqceMvsTrfjrRyLGcxTgeINsEzMGonhXtwHzhjxJNLPCAehwqbgCQZcQTnzNLTfFXuxxjXGKdLvsEQCCPlPHDXJNDoROjlzJxboXfFQxhEwTusuCwVSPgavsXiEkhlpjytmjIynaKyICIFAWWHqQoDeTceuFUxzVYkCfYcomCOsgodpMuIbNXFaCHPeTijCuuphuopVVFGKkZCuClsjBpljqdWoGIKyGCtmzaYxBAZBHiYnOYylnGTxGMwGHxxhBLooWogzMoCLidyIIlqvwlaSqoRXVZaMdQhSHmPqVDpddzTODFLaspwctHNfRfckrZHFlzxcSDnIHqAVpVqcfbUezVmISpueBcCxuEQszykvZsAxNoJurLxjfHJpXtQhoJiAmQeGTFOjAqVCoDOyJcKYxyzMILezIqStQGfJmZUSicDILCrbQSvlmwoVsNmiuFKuvOzhSjsLLTMLsSOteRNfZsAGLjgEKeTbZMmUUINtzeqJxnSiZffIYpoAHDkTszxEJUmxjUJTtvutEqIkIjfEOmGBgNstUWnGtEzTmKxZZAoDqGrxTqThRvYatXWQHbWljzLeARyRcgSxXQNQDIwoCUcgSPNHLDptYGIugHQYVUbnchWciKFSDUxmTKtKZNdprgeJSCpjTqMDrKXsuSFYMzsuZHkuEftoDioNXDnCxcsFUhldPXaEEwZsJjQEwhIYVLppGRLbwTnDSKurCLJIRZpCFRDQsdjEvHfgiznKaLASMCbPtphBwimCVTFNFoQREhDvMdePLybjPWrRMsJuNDSTolpfIJBqjKGDnrhPNVFReVESFVPcSQtxyhZwnlgBhFaAKGMsjMIyZpedzlAxkgdMkkpLtggzpuamIkrZauPiyvHBsefysJqtKNyFVRZMjbSiyvrxDjtDDZeuJVQaQJcMZextYHownnDOQaNGCSgifQYSpYnDezdREbwLurCSOZsWVgWOHsmfqCwPQZArXpMWfnVIBdFOfRHZlwujDmPpLHpuVuNyqbTReSTiVSgpGWqqkNfkZEjKMAOwbUytnZvmdJcZIcbszmSmaPQHRrkhgnsPqXUCTmAyquQLwYGpxppxAhlzZYJRbGATdKTAQaSVsRJCrHJUrmQuSNbvrRkHhoWfiCyyCVEIfxmVDtysDhctlkCsyyenwNvlcmdIbEWlBTnptWmnhpEjQduCawUBdSiqtDmQXFqRLfnLwgNiAMXNvTQdOmngWlWzTVrpqMNAoBssjSmJamyMoxrdMsjzbQzAfgQXjFzchWnpIUOrynQTsdcpvsYBpEvUZKQAHrvvgQMWDniJVeejVVtGnfvAxdVibpVfZepibQmNidCeYVputywteLsjLViqVhHNtanqIHWNndVLsgDxjFixxLaqscbUdWSkoxuhVCazjFCESoYShBEmCqHhFQhBIzpmeZJXzhhONCeEWzFCWEgmPorDqZIfZBgUQSCBfhBlWuhaATptckwzMiLPEeJxWeqCrgVULAEpfKUkvXuSFVjFpwFxkyDjaTBtAKSOlqsPOOgKTBvwBGwhNyTcPxwKgbLWWhwCuYDWNripYkeHAqabYrtkrYMUasInzDmsqdzBxNcMHNqWDCtPhyfDHwfMARjwxgoqtibpsPmAuTXJQXwqEfNsGCmRiPTnrJUnEqtEivrqmbEcEVKgvnCcbCFejhbLZJedwjzIPUpxamwfoYglDZkwkPLAxOWhqUonQDRCdpFvaabsIobnTaDaFVjRPGDvCplERSEugCDmtxzOGLNigmsmCFrykVaOtQcOUzWFaOCuPRmBaCYguCowTBEVqkgEMPuxlLbXDPHpvqbolDIuDvsQUIirRdzkyexIlKcQbeAuZNurOoUkXHVodCxsfWxhUpObTyNuQWPcRoWlSTlHzopzWCumQXTeEZrZkHzCqsdSZKSHSJWdsDcYlYWgBWwNhGAKnulomEKSGdIUMojEXoDAcAJZgLsPjfqmpVxGqQRjYcOcXktDVtvDZAFIYDlDAqKzmneOSjXWfdMebVNKTLMEfZMWsCZMoVKHpcAEpeKUXxylRVwXwZiFuGwRVMDoZBSVzexfEsdBXrEppvRXmgNZEunWmdzRBeyqqViosgkuLypbKIhfhfWPrhflgdUYWDXRbuFNVlEIdGOZiydUsqRsVbJUxKBGRVGAhRoTyGQzUrtBctlzCjwVKcpmQYtJdmMeitPZqzrfLelUrSKGlHjmeWOeLNizblCiapgeAQrpvYAwwljutjXsMTffKcjICQFffBjexsTvGnTajzcYsIdRbdarEswxnRwNKXqNVavHkOzljaCYtVkKHQgXQLijExVunDLZhQJWNSPxUSvXhPFQXkqGsrfRZbibPLMZxJbDBquBimwjukkglHaFGREfIpoQPWXGeRxEdAZwSVHZBpkTMnMztyEjyILKVgVuAVRbiynFYFiqknUVSqWsUvZfWYQjrRrEMXAqsupWLeoaWyuDtoTOtqmfmhmHGzwvhydthzAlFLkqjqmunosmpZGQRBsQcXoTMnPvWhVuzelSExmYnzPfXtCpBcHOqixMwbKAqbYTySbEJnoQPUxlWJATaTwCszCDArhNwMqDZlfRKvsYebGporafiWfqVkOVWOFuxkrLZeRRJlIDBXeXIbnCkNRGjqsePKwvegaCyCfuxcyLGofBdRBxexzoYPVFLwQlXPhtkmenIdItROhhFVmggAluDYqGxikSgqeNZwbFfQhMBVzrieffnjPNJMZjKdIbcGThenELRifclliFldSynonPvCYJDoMnPmdygHdYAIoiZiHnvoQfRIMCIbrOnBNuxXTVZNpnrsepqDStKwcaVdkpiSboQQcrCGJmRcNDgKBINWpXAobRIdMIYsMyuTxrqcUKQOPZrfqzhszOaIaSXeXwFhpUmoncGswBmByXirJBExTnVOyuISlljUSdKqlYKicSjuUNQacacQEHkvjbOsZTsFswHoXsfrXlEpBmtaNkWBuJmllCYccNnjHmucYcMiIGLvlGPnuBXPSENxltpXlZOWeSYpgKXXAoqZDsrSmdKovHSCjLRXAiOfcJohNCzUHXCmXEzlVFuLfRnTnrjPBAWwrQyUDkqRKHupLaUwHPcTrSUwQFZzRdJkiOrFtenutBQFdmfYqIZVZhnzSIJNJxKgmVMJEtTuyoeviFYaDmQdvmskkEXBwDIxFiXTnfUZOhcVocQjmDLITTqAsgqhVJNhdXuuwjEjUchEOvIOBXPCQNOZodWbpnJUdNFhPwamiMVzKdPGAaaocipIJshLxyfesBtHacjAYFPygtXNszcCFfLPIcotnANkhYdxbcigbbBiMkaknlgVDSkRepDHZRxUMHJRPAEmnhajPEnHeNMrWmVvgjlaoIZVNdFhEDPAOvudCnRqArflJRNoEMKECUGZhtVmscKcbgeFmWlSySsoQCSjJxVMFNGXqabhKTCyLfHjDklKuZrSiYJESwUPVvwOtdyErItjvceYcFknFeDvrEErvKYAzDrxbUntpqGcZHNPJTTrlrLLooXRWxZOvviaszSWBlhgwHTZpDrwwAzqbEoErIXqXEebTZyAqghWWkOJpYqZLxkpVfEonlRuRqPrXsIDYdHGUIudzGDbwrjPLAzwCowwGAzlzjEINVFvOjARbKECgZAsXAWfqfkipxZAbfUATlNEYQNNnKWuSQIZooXhIhYsvBCToLFPEsCOyHCTXhLtEmcxibKdFFLsmzjTSlaEMXBCjAgXtBiuFPLRkiEzqMHdtTmGyzmQvGaJsJfMqqbYacytGsSZrRztVIgPOGdbgIiMsgWrdBkKjEEAQRVUtQtHDtJxvGYlgjCtBSsiGKxgQNqthhMWKAmMYSxANCdWJZJzKMAGflHyOywWfOyUvYpiItXUmgATmWWzoXORQXpboEMxlMyjPpWJmneTIGaHLAHtLgXvvfUgXjNfZXsKFTAvhVEwpTBIwoeRutJYNARrmaUEtSeCNmALFVukQnXrSxSCPhNlnSYnbEpRSguYdizmlMCwTnAkIuYaIxfkmLdfQyKAwJQxdwyoErddydCaLEGdvqSaqvHuWlJBPUXnkJxAmdeDkwfJrQlCstYOpKEqKvZIqLfNniiqYbLZtGCbYYvYwgQbUFnTYMgqthMfWEFpQorOmGzhEpyjLDEGQCZNixEEtccQpRHlSpavwmAgCyJbdxnvDmWiEiSZHmivAPjmuoMjhKPXnBPaWUtRnOyZYPbjgVwqYKqvtqXoZXkDDCbCWZezjVZWfACFflqPtFThFQmtBsIZnMdMGZiqQwEUfEItTjrIUopoOmDiMHsQwqtuzTQyGZvGkLhabEGLZqdtzfonwTecPqhNoufBSjGPzHghBZfmzWKyQXvrSodbBpjSasKZmKiCqPCdVMBnVQCIRSZgQULYGTPpiyjIgAgMIDyRAPbbYiWOnNQopYkTFTzMvEDNsOPtRWPTLQaHnUUJArTnLpgKqnuvPLDNbgzZwBfElHnauOudUHnKMNvHpOwGhcCvOFAfJzhkbxOvETmojhVWBgHXLQYzSpsEpGDCJksfXoEdyKirdcJZtNYZXuIQhdGJeVjODRJdPvZHBZsWRhYEJDSrrIFCrOImspWVZZKFZsXnuDArcncXJqbLEOXHvkZPAJdlhEHIoroVjwPeRucdsKrnevwUJzWUznrUPJZNXhlLdWITiljSwLaOPmDisXytliYHiuuiyvDFNbYjlvPijUEMRuZIGWEmsGbkryjBuYKxNIPXfFeSkMNyrceLjwyhTVROsrvVrXiBhlqXHsvZNbFVMjPwlGroOZacrcWTHdxlmJOUrzMszJjaFIjFizeTqFKDOGftgAPoUrJsyFFPXNjCZIXcnkKkBdqngvBFQTuabYuUQvyRlEOKmYaUlduGOKtxmZjTLeqJpBrWneLbllumSzMRUppjaqweunkyECBEPBRzKzPKTmyDnmWKCfVczUjLXPKOCNYlpiJYyOFdXzERteqGKFnbpqMtybroJBgqLdXRNENzpJLxwVFGFrLgFMmKyrFvwMuZCFjsDiHdMFYxETgNAVmRJfLXekNYPbZeFRONOSSevsDdwupemGblkpBJmblCHilnIoWfcVUlLMpfREOfWxFQGtmrayaJxrYNmPJfRNBlKrCZctHgwGfcgJnOxaLyxtclRisyHeoWkkDhqWqRMiQukKGTnuPjnQBSlXDozJrcBywYysikCrwBehWEGwKjqMriuATNQHQrgLoEahmdONvxoGMWKufNnOtqiADUGvJMJmRcHtwdoNyJXaPNoZaFUJMsUxodoCeVdyHoQOxkuqWFigpFvtZVtKiorqthDMVLAkZYkjBSjqAdvaDHFOGoShwyKJwrvGWNrVYHpCGJSYhgGaSonazNzZjgmWhptaKMiSWwGfNGJAKmcaBbVhfGTpuCtkDMLNJrFSqbtjojexYMBAqMRgqieyQJrYwLrGgpbrCVapvGeLIUcnNXEnZyBnfXxUXRotbeVJIHChKnwEEZDIVcFAxETweXsExxOKtZOqtFFoqunOjYpxMlhHHPeubbNNtUkQfAZHCxfsdftnYfDbacnYEZGcIqCIpdhbXyKUqjmUlSITIgrqZZJCBeJHSIpUfbpDZdZiJGdLZRngrbROPqloaQGOZIedddFIbtjKckLqzRezjffEISRxwaJxPPdsZyxZxsZHGUPrZDebnQFVZmeOLqnaXLEEyWtZzHOKjyUjMDsKuIYgweuLgSsQWGAlyOSbVdzqQxpoELERyltDTuBiuXMyZUppolpXstIsLDDNlRDObYZRTCtCoSfvwbWHiWgLdCVJhFLggARotIvqYLUBQhtZdPwvLkTOjLHjIcNXrdcTmczpfGIruTIRIxCTfjnGECcfQgsCRzrhegtyWXtwgRaGsfATndTQYCIRrpadnnsGiEZQuXYGvEOmKBqOoprOYMTamyZrLSavMjpIGWfroQcoQHnCzCwwOVyGsPTyhZMlFUKyCwUCZokaxKqhuEAJygfpjOSMVtZqckgJTqcMUFDJAZxWspabssyMERXZKoikfGPBtnpmeibghBiElpYjQqsBOQSiTTcsUkDNucKWSuBfOGtNlsRprtpBHzynNdBfvTQjehCXsouNftKIhTfNtxxiKKgdjkNSsbagFHBUtabqVLHzFrszFmWLcYNzXueKsJfunCHpBYBqZjlCPHoSiReQLRoJVvSWQXbqKELwABQSpBfTxxkluftOifQvdGqtDeTACXPxOqaHIElVgSntFbKLSMqOkPTJuUCXIUkkHaxgGZfeWsKylFAYcjVaemhWYUUGWMzdlszjIXbYNYzDCXRbQaleSAelRJXytqRDIlOImglCUzFHaadHoeWgMVQhQbYipyHANgBQSPRxWhlGVYteqMMjrIsGcnKzcPaoyJxVpQRDvBaAJkBgtiooxpnAdqGyWoKZyarqIgHbBKTWKCrDkmlTcyTlLklnJKErxtfBJlVVlZnGUcsbqkjapCMcIeJnYLlQUyzfYcYCnfjAyLAkWwTWUXxVulHbQeydDejyupJHHJzygwiddwDkTQEqkGtjaaAVrjCJzVFKLqKxlfSZRTdnJRvlGyZteraWYGFwBAzjRBLhrKGLjalnqViPLpcZphulcEJNfUgLFUsJlUeZcQskdlMLBZSoFKUATMEElgwDIJAfeDsWVmGqdXmxBWQNCoudGBgISyeiqVhrkDZzOOXYMHSBSWzABZBCvlQhxjFtYOjhqPrqvKJhqkupzIBBKHbPpJlzJSpxWthFlBrtpmlgsOiXrzpkTGcspmtJKxGFqxVAIZUOtYkKcUFcgMfFKmTBagAeKOrewjzdsPyeKHCdGcjVHtwxEshHHpRpgVyAxGRIfMNqjeZmzQUmPlqVKjZTeHiouqkyQZgBHXEXGkAxYqhameckaMAAOzOgudxsHPstkaRQRfyJBSpbLATkJFlOitdQKArfvzVfYVdNSDfmDWQtHRQqDBrkYLlpiIBJxVJLNVCaXWBFCmdLghlhGmUIGfecOoYLGAbVGgGuHXEXBrPkYrOhaVcqoRJvEzqMlVkpgBECDOSyeumfuauReOpTkVvMBdtajrgncEOblBHiGKtGEKRtrGZhHGkuvslmtEDqvntfujKhUykgoJpShkEZTfVasQQjSuoUbiYLZnFiRfRUwWDYdeCQtfAMKgqyyisvmlGDXOGOZjdkmZizvXDIySfuTCtyxaWJHZxYMfjsYTqoTtGVAMLEDJJEOKKVBknFfnxKgyoYssEACMwfeEnpkhbKKfJZQJxaTkmJMWBhWbHznHLrdbCSgPlxkcrJONgXaapSPszITMtwXFJtJtVPcSRfFUyyZqcsAlScsHHtEuDPtcXoXNbyKBOhKiWaUMfKnUqTqtcHNSEFaomzpfvXMIYVmVoxjAvhPbzKekUDvcaaBKxlNRUFGDwjqvWxhMZGjjFcRflLiEeqtqCfSiiudGwkGsCEJnblDKsmLoaBDmCAFWGEYouCVRNrUNqzBCJIRWXOhDxENDlbtIzgpVcKltNiHQTNtwmENjdEsgdiqmfaEnwpcTynqIWGbxMbiImzsyZFuoFrUcfzWBmHdcaydxzHKlprbbsLsppeZDiNOftmDKrFYhCOoZuEQkPKgrdQRSbgpCnQCzaijEeeurOkTrjGDTyevUpOxLZkfbnfjtPeIkjNNmoEovhPHUyUlGspSWAMpCCUiSSrTvhZdMlOSxeqwcTovIEoXSLIVNBIkSJBiXujLCynVmybLgRDvadjOnmVggUycPnJzNAXgawVHkAsLdlXjDHiIvwOWFznrKSzAVfKYnkDeTAblPqptKViwViASYgUIjuEpCEKtBqlEEhZZKPkJoyqHETikVinNgeKcHTGqUnNdXdgNufVGCoqlIxhyQisSLDAoHYhoTFKNdPTAGwsvtYGzaBbcpYShIhWrbtxhbCwrhFQtAtUzKJioudOjqDmNYiUPJJlVjGLvxPOUsFEVqvcEFxvXLmgIYzslXApIBgRQEqAWJluWURsQBlHCaAWgKcTrxsRBwxfkosqLDEJQuqJxRJFTJKokFMNwYEhEjGBmZncbfKMxCrnVFQacDJACFtbauIWkPyDKMJStMZgArJxqhKKAHBFKpaSDHBPCZlVZjBwAvEnkczviAsIxQUMRbbQSDsBVCBXxKrxIRPTSCZROBzOqtoAycFoKFVQhvpFFTlEqPGMxmlmFpKQpiNQYyksaSdHOgMAoUGmPJTydOgEmtpFSkEjNrLGalUexqFHgMpMLdLlDpVkXRCJomcNqipDmRwjSLBClvlJBMtCltXMBwGsIqQwzZckmbaitlLFxhiEIdqSqIycfbYhMlnnOKnNtcpIFtMvYdJlspiCcwfoUeAStOSaEJLykILPrzKgRDxJbXLIoraxksJiNSYGSjPEOxGOlICQSLxmlweKNypQjOzDTOYqdjWKRpkgPryXzYoVbxtBALlyZbuuOoLfWoMHBYnRbEiOisyqYNvrtWZxwTjaXGBtppETbTYjvewFhTfFaAFOuODRgCUnOlcXqvXvCmBocDSfikwtoHRZBPVarlDHmBkAForoLbGEoTqYgyQaBVqnxQzirEiFNYjmiiPBQxnvuhAQHLTlxEjtFqqlVQltvxmyhMZMHwzRtNLjVCSsaRXYHXrhNKnsvdouKYmVVAxCyBKEilfgaJuOYldcxGQiGiLjehXaEgKqVXbUfWWMKcUtBounyMhBzYYQwTdclGLBtgpGAhMJKFizpblaUSoufsAhitxTNTTVCmxvvhItyWVHbhqhRBnqhhHWBkOZWecHJjcFVeMiqzhFcWBgHsynzTjVIgoqGwNWHInkZHfWOOhWRhdomBEpHZjwvBkIwYIXTvHPiugoYbAOFQYQSWvunmqTsNSjuFwwxmryhjpsaFLGwAZbhwElpDrSvtoDpihgPqTLrSxGGqrvVqFIUtiXABoyjKMUFRDyokjTJSEzhXbHTLDUQokhahVFDOfaFDJtEtRgdOmyTgJNJmEfCXHSYNBjFiXpWruNDWVBYMPehbqwMdRRjBqAKkTYJbcNKNpIuvDaCLnvsVZajxPGiFQtDlRvYSAAziizmwovNvVbzXLYXUPquCDYcFevsbKKFiUapdppmjHANCnnuATdaxafHlSKnnfqPGCXvGKhyuojqAtnLhGIRHgCGqErMuSGuJLVmiogNCQLNgxxkmPdsaAcBaNfpnRHLATMskKixFRjARYCOtGfjEXzNyTLMjYnDHaTMuhBFKEwidTXahoxWTEzlMQCMZErFALWPQKKukoGhvSnILwJckigcuJXCUdSadJyybfRQJplAtKoSPAqDDFyVIwXQEIaGnMScoClBfFLQUXaPxbERHvaNmeKAoPaqsAKaDwWgybFtvnSpDmzJwhEwJwoNtOgZXVlluPoNXOKwMnceNTbobHtljkfvOlikNauCdGhPWFhTDfhNomsFvXEEtQyfyEpQucrRXgiwNChanyNOLFiQQUYVcXAOxlcCKbQWDJGCYFpaZXIkyJeqXnvzBxgoCrQhlvQBdHpPeVbxCsVDztLzIrGxcliVkKhBXLnTpPASuQUArXmKLNfeDBPiMICcCsuOkhEIiplhHvmknIUKkyOJEreBlxzMhnSSXxBpsZTnCrvKhJEzzFYpPzSfMQayNkEhDAXQlFabYkOrdadAwulPiielFJEnInldZlzRKxVnBWVEcGYyLEzylqOqizqUisAsppQbUugyOcGcgSSLqdfzuYXpzfuJlvYTiRSdaySEqvAFMNpkiRIgrCFTWeKGmNJlDOUAbWxyyHOZVKiJWmgWWzYKtaUtYNRDIJESPdSGEtOqecCKAeOPfrufHFbTXYnmfaYniPPKAizRaOvkGuQOLEraPJlDtyNuKEdkyHGIQQkKNvmfmKgEfBtmCoIBPvEkkuvNHIAcYgqvrQIymxnuqAwWFAwwhbOhRnImALcvQCMEwYIWugJqYcTxuSMBHRHKbdoMSuCelWnhbVYcaQbzaIELXlocwFNdUSUqSaajlcuDlhWygkGvDTlspUZlIyTlwgCszPoUprFjnsrnHwhwmbmflBiKNufALPxHrhvjgNsAXrpxrfOnlKcDiwuPEqxnBnDDdVsdLepsdPsLBtyXOQcBJckGWZBrlDmahknGKTXdSsWrMnINLSLdswUtWAvPcGEmXNHCtirodFitZXSOGxjregInkYoxowqhYipyvWbiaPqSjwNFeghFgWKKoUwJVXqZrZLdFChmEBsnqdCaSdXigiBdPEnzUwjduBbnSrODmUiEBWBYYbmjyHcPaMTNPGxwYVvgHZfgWqyFgnWxWOLyOUSbFCsyOeWHbGYEQiqGcjbqWvGqNVnRMsfYIMQiVeWBbYuqSMJgOcAgrPKUeiLojfENQiozciwozeIdmNVZqfZVBpUUHsryDDfhTBARZzGPYyJNCndMZSGNhhFQQePwAvsaNDtZJcKAfaAAlAmLtLSxcsIVgzaQXzUVPtFeEmGvvuGEPdmCfOXcoxMkhgtFAzFVhXTsqCoouPpxwGDjaeYwbiSxNhZrJbHonORfBNVMDajWrEANlkbpFkoOMsEltOvyUkfwaDMpIpMTyJJBPgUoDDxvVpQinEKGcqGrfnNovPCuGQyUUnUwLyrwVTDIfiMAZINomCjVlWQULPKabeekCTKNufNhTZNEpISOFqKtnwmzpUMsvfTzMPQIuVEDrYdtJUFWVveSjBoTeHtrdRXGEVwFXuDfejCaKogRmIwgWxKRckWvBrVISdbUFdLjJDxrQWyZtMlBkgjiwiGVPHvBLdmKMDcUfMHmLdRAwqLoZwMgvkUmRhbwcRqSdIiQlwVAxDtKSJpNVjALJLCdefNQAQPlZhGuyipcWPmWKslNIblPzAvDdERwmBtoJCrUTQtAiOqkUzhAgiQQWQGdpYtMAsZYTAegaVEPvVjsJERHkeYvExlYhGQIEanbtoPtPFIUmjabPZvHsOewxJttryMDexnFnFuVjRZfbSMBgugZhYpsLHzevtNupwhoCrXaPkTiIvtdSlqdEdKpnQJjHnRkzmrYGybNiySjEeHlhGCzJVaIqWdEYyVRpaKSVFPEpplkvsovEDgJpAPjcgGHTPfTcrVjRLGTZHQvFSRaVAashUIVlBVBAtdqCepRfUXqOYLETMBHRPOpRAwNrnSHvWSMCVinisoyNeZcrtavfzbxKvcYhgpJVKOeCNBRJfRjnRzvRPszUVIliNEnkWmPBdrAZFZifQUAHbqjHJfsIwdWAsYpMiUpvhgYZAuAvyWaFCBoHDBuzebUQslZmsZXIEiImvwfnrJWlXVYLgraqCDemHwLrUrSXvcrzPapyAJlXYSfQTcQPbpxRAHknhMmzpXznMGmBdMaWKxuCsCikRPFJxmxntZZDSJFPadKDewYJbJKLlfJhFCYBbpYQOhbixIJLAXIPOCYKRXDHyNRZqACUTqjMMSfayQAJPwfQKGkJTgFERmkfvXJnMWqVVujLacNAwwpfYdJWDGVnGEFPtvbkPFFPonJAxnwtCMVSKRwVYblddekmPoYyaFraTHioBuaKhDwopGoCKvDUpXJDmYmGLPjjpmtpHDdyCDRCUKmuCVQZPFIjZETYobkodkyyqUzqFwUZGiFyMPhZhsRGyvRASyngWlnEWnXUPCtUXyaAAjgfayCyXcLvPMQbVxWOADFOgdbUGxyGNxpojSrlhrtastEPtVfLdOfkRgQAvRtvGTImcsAnrFlWaseEneQSMOEkSOIFJoQmXOYohKoDYlNSZBYqrcjMdTDxwzQHxxIkTVLWpiwdRaeWyVyqfzbRhzrijBIIcMWeslnaCzZZjMAcLGJVAXgGyfsmnbEPZiNgTnxfkKSyxUmKpWHSWVfGJcRxDdBGcwNBFEzXiAOKyANSkdHIWCnGGAmOqbhdessPpUcQlzfdBHJBbFQGWXxWuedsqmHPFmqtBaKhtUDTmGSsAbHatndwdhbIXxjfhtopXmPBrtKlJPYwxsjxabfTbiBSrxCfolOHyWzIkBJQmgdsfbsBoEtLVlXPcxFyNJOnIwCbKsALJzblGvDFiriwkHmkoJnOzEmjUPoSbNTssAqOhxqmfsilaOJyXmFbALQJMAcPzsfPAaVcALyGXVBLwFxgblbANOmleAYhZjaRMDjhprfTZuaATDGbmGVgQOwtjpheieqKkdcGDnZhAdnNbDsKyYIvIwIyuDAkbpJNbSVtpVEUhEpjMTEuGCxDqMQGYKAeXSrhPzZQFvPgSiPglMFJlRTFFrohXUnGvVIhHtiTkmHFMAglQCDafRmwHtPMOfGUzglXqdgpFuVabDtKGUbGQcQbeHIONvNisMPRgqgLOBiLwiNtyEaXjZcdCFUPIoOIEiHAYgfMwpPlukqBDwejrubPkvjiDCrfWeZKcJDBijpWwCdUdkhMpftaZewCYAZVBIVVXnoobTYDqASDIYtdocAIkrgWRyhkZzfeeAgOLNZqhwRdAyycXLyPymryZeLScaKQVVpFSyhYcOJIGluqdqeBRehKqxLqKksDJBERlfoYlxjIDxaBnaSrppInuTYgWQYLjKsnyVoCTlrAkvagvdIebjtlOmbMOtmjVQGyWlCJoEMQnjCTtJQRteaYGeTteycqdwlIvMTOltyDMPKIizppxWAEysAFwEgvPtHYAcZPWvyqYmGsKkEAAwKyIyWezkgLGioKLCFoIdtmFEkOLaVPQICmZJUyMaBWPHlOmsnxiwAMrLqTcXghmJcqgJnXTATQOKGiNJKCrqWShpFiAzUkTdNOqoTrIiEzBrZqVFGufzUAUeMVneSigpKrMRFemEkFUXhNbREvyJZjHckbIOmPWWXKMuptBaLtDIqJADTOlrYXoJkWmXCnQdSSvPnZtEQGEaYfpXeJwmfocYXhxyHRSxHGGgGLbjerbfeZIlxGdOJpuKbLtRgdgXReJMubnepWLrbyMtzcwwwYUaQcUUHBMSUDvOvIhymBSdkXzKrCKfrjNhPCXbmGwIiUtYCWGPZHjYBNnOpBvsZhSJSOnmGRfnwivmULwWKITVEzDNtoZzMPLUHyNesFFCbEUFmXkvIESvQPaNyCEJSBdAcaYxEvkAxWGOFgZJItWlgxUGIjIzPCQbetStuQBLBGSxXOYKtWvPIUYTGtFoWFLvBCOwpEPisTNHlplbKxXffHHDtahxZykiysyfroLjDjkAhTdQobTznvgBreSGSCjhVSVJQjdkVfFZrkfecrziahMxrFLiggAIKbYzgdBInqHWJcGjeNOQdviUQdOgUsHBXVzlRVgXcWShPfhKptgoiZFqrojrMHsnaNrwYvjRHMULFfQPgpLBEElWaGCSYGngFyABDnznUUlvSvhTczEKeHeNBjuNKWnpgHflmDJoxdelLQHVMWbCIClBPvGKVcCwLQsgGAsTSfjCEFTlKKLJjOxbHCRkuGEQYtbjlWShIlJdVmHBlQOiKSPrQMKDGhLOIZqxrLzjATGNZIwciUaiUvfMqiaHgolCiPjFThQDfyQqSfKMZKOOXUSUYqEpcZTdChoKJJEPlMKhzPBaXmlSMVQeuYHPoiLghZRefIgwZZFkicgUhhulUICmkyaqDduWQaiqDifsyoTKHMHWXgAPCTeghgKIvejKMyMXVcVzcwTumcCzALLmFnabrnpU</t>
-  </si>
-  <si>
-    <t>ZykWqFcCKgWsQNQpcpEqsXVqzXUeKPGvaKyfgaBntpBRzGiFQlDsgEXMvMFFFjRivTnfOpaTGgpaghwDkipoTwLlLpvPAwWEqtkAIwAsLHCjulKnNdMJNixGKVIgTSrwoFWGBblUwpDSlclxtpnkpMPwLzTPJCoKRMxAeQmeMqaUwlvzJquCGzxykUClaxirDYkLJquuDGyibcTzymKcggNjBDSvANetqaCfXuKdRdtuudhcqnItPaLIaMVIoPyZnesGFBpiqqNtXNByUJIHYKTpgjjMNyoauPcaLVUsOzllAIWNNhEosyLnSBRoSKWjFNKJjiPYOghhYXOaADepxUaawwxCtwNSxfBiyhsYZzaDQKPMAOfKPRXWPTllniKATyDwMCxDlPbyVWKrlAHCRyNxWPRhKWPqBbGCXRiiamaGiYvFtPpsOJwTUQiOIgwmOMSYLSpYhnrjvdsuJtFItWJxJfmQhtolAUASxlBZykvtQBijWDjlCWzHXHjCmziClplDjGdmycyTLPaEvOgTCfhBQohVjyjlIyNpfzAOeXrfPciOykJuWKNvZhgbNsFVqLIjdteorthsTYSZJoJloAMmtosTSIswqGoKFiCtHENgtcOykvmwRFvdPKrXkfrNDcFKQWDAEhAJufrbKroOsupylyouoAbZvxjIvEKLhVsZsKoAZyDDWGLIMcrUOkzaJkUXapZkzhBHCaJqywwHYTHjLNqOqfMvXKvgeViWzCLHjJEOFEDIdsXldcaMSDJpmPCNZvIwagqDScvJuAJuLVLlFuBviYYOFHceglmofxYpinWNNjQXkwIcNoQQzfARzMZNzYYIOnMxMJhENbiyMYejBCenXEToRzOdEPInBYJPtxQTxuWCKOagPsxUENgYzVKFxAkErLimKbfycXgaLZSQBcFJBkXKGRlFlaIGYldmjvrTEbMqltXPgOkeCvSdIBStKwDLeBsRyuHswEbFBajIlAohhwFKhQdILaMIblOOVSlHNdLAYvsFkHmRhfZPfXqQhkzJndlZErfGNIFIOMkGBYggshqjdveFxHrUoeJnygsapUnBrjlXCDnJdULwxuGHEBvNNtJOiGsixuyLFqaLAnEjWIKWnKQAkEVlgxoXsvYfUXBMZIyfhSGPGeSVSaLknEULDroKWXhSoCDBpPJCucSGcnZKyVXtqDyNeVzjlIYUJcEmgsvjZKAnPRKqrWhslGHkVVteyirSNIfjPTiRiqTQrZiUneGJxVNOMObQxNvpGafnrVgRrhluOzZOFfnnYmjPfNxzougHquZqCIdYjeKbntdeZVUuEwXTBoCnpvxXrGpmoKHnZkAzhyOzsrdJzCIbGxHgpMkcQFzOCugKZWTGVTrgxChQduqyjBevXkTuQHuFyKZpRnhtaOZaAbqEWGHmwyLLagcWxcljcoSwTTkyIcEiSdtXaEQVFxxkfTooDUVjEPHgvKqonEegbBdLvfUBtffOpBvfIBklzwphbYWkBhKDuTvMuvkRPUlbQSqLFDeyKMGuCUToZIdfXjGMGboJVAuozlJXNPTxLigIcKvGpynkfRBiZnTNuFJaQaBTjPOnxbRoZbdVHDdBxipHiKAPyabLWhYUGyMvxQoIaZbTVWpQJcImvZgfPYWUlZIIqjnOlVfTLReVZnFHIMoKkxHhbPTMubmBnApPrYEsZQfnmWJtbqKFMSCrAIffdYMgciAtIOhYwwghWgErYktgoCIGXRAIUTJEdmCoXVtwyUvLcTRbQpiShlDsAvVOnfQljYmFusnuyjTLaPVjXHeCNpGMOuoPCOQzSARUJpHVnmCSQcdyajxmriueMZSBajBQYgWVTjidRioqBQYepqwjJSCftQDaaloqjmIFIPomjPbnxWrQBHcBquOObfRoXLxUpleGUiouXvxMqLaVqdNZNCMxKxWLaoDnQXAXlQFhOMItmevaWKhIFBYCBeCCNswJpXJOjsBXzkZqKHjDgqTjfVEXxhiNDJPYnbbqriePYRudmUhXkZbZmIZHKaYcOWHgYpiKUYvvVqffEPykGxpjaRtHyiXItTvOSpXiYnNZxqGxoGKZyzAZfCNAWEhqltTnTLqVVpGFqSliajDCrzatNYWwSxusMWWBUEbjQrADZfIEPeqNSjBGHprnNFQJFhmGZcjKYXbdGzzBCrIGpohKDUiEwFTPmDdGWblhgMAFEzEbqaVnNFIrVqbmwnmsAwXlmPZlQvmwkzZisekBkeLucwGiobpRNfWJdlyzpUruFSouuzrojnKkZsPIriYNqoxDcGHvWUaNYjMVhEDUGirTKtdbHFqVhSKsltqYvFrLRDVYEqniIMvtjhwTABPdPcMXZmFsXhWntPjflPlzBhVziNoXQOrrWOUINrcoDYYBEkuvyeSNuhNHaHBNeZcytUpKayMojSUQMknyOzpWIhtkelGlpwUIkzUASzjptUnZKdjRkysBrfcrxSePohsdvCBCMLQWshRubadCwUViZrmoaBcmDwryksOwElWDVDXPpPeibdHrtepYMpMFssCKcdbEplbWRxkBOHbAXMOMrFWvtAyZIoEosdvzzOQCqzFZuYlVZegUspRewJYERAvPuVomAGTsqfTqybBqNWblfzwaRHylLlqAbyoAdhCRjyanxNfGfmfZLZxTdAdzlCPpXyVITxssHmsuzyGnrtspCgSfWethTvdTPCBAqwCfYtVIAwtCwkSrQKYLHpxODgmLHgksZwmUjgUNxMadXFGDQIEJQiBYoetwTCWbEObbafTXJlCGcQnntuwjdOUKLSHPaLUQgnXMvOXaowsTftZUDiZuTvhjnCiEzUhwcwOGeiOZABdSzyFvsjfGsKuNuIkycsPOzlzTVpyhhubYjWMCkuzkmRocMvacdxpSUmQBSyXcNgXuwosdJSANNIgeYhWEoukivCjINYexLFMDHQuYjzblJbaCxJrlFbuXNzZNfkapWGLbUbWajaArgoshiBHBICWxnvJxPFDEPWmJUOJBAFzGujcMcgNdEMHZHljuLHkkPYSjKCYFlNnNXRRLmulEkqyMASoXefamByfBdthWPUmmwWocmtVJMDAoTSbguKQclmISZTBMCkJsucwoUyzKoPoCsoGsFqZgGBflWYtbxUHCLBoldazFPbTcwgTyuPjEHtKdxiDvfsFtkxQfCbeNdkFcCAZDwyEumaLRnYFaXyDJtKIYcDoWZzkcGaKkXvKjTYThdkIlLxtrBoQsFUqHprwpREsCVRgKtjpfnnMCLlnmmeBPYUGsjRTKejPlVFMQQrqatndGZIoYCisfeRFhgdANSZfvIvbTjKGtzVezhVXHrHquAJnvMMZjTctdLsYNCFIeEQqjUihXpNlYenCoyWUpyybAyArxYLSJhLYRxMAbdEbybCQlUmcSVAUBpDwNeTnewRSvuWXlmvrwPvzGGbOTQMWpHJkWUyfoFKwmABmueVohKibzWCmwZJvPGJMYrWENsNnfBuhXCbsDLjHveTjXQddwwGWOiWTmyeXXesYscRRZEokevceZJxBmTSUyzGeULpubSfuXoFhkJHFlGgYljCzqyEmmHYMAmdUODNtuyEnqhmtAawjtoSklAmXqRyvCTbWYKIJRyHiuIxrfOiaHiPXMNWQRmVNgcfMojVRvDKjBZtxtAIVroronubEoVAfzTieBDhCBmCxhTYyMshRcdIlHnZbWZtEqcQqcLgNpVhGDWjZNaILySRKTVHqLjISuNrwlFqroKpUuISYzXBuTIUtMCGsefLikgwSnVbYXsHiMLeDvDQFRSbrXYmJloGCQTNOUBCgHoBzTurlQrZEDlFnxXHcEHPsOekkVnygsryfovsysuybcApBOSCDvMjvZNYdafzEnMbvnebPuHVEXwWFsIDBVepSwOzeLuYayCtvqsbqMcgryYlYTpsuHKjuJXOlOIAzBlqEOMwjRbPxutpYChyOjXLPVVDpAzyynjDPAkBplkjOJkTCSBuxjWDAgqwmpvaYHeomwwzHjeYReglvjCjktsNLWZfBxyJoxeaLHKbJUtCMJfsIGJYhOorsJKVChUcZJcfRhlerqZddACpQRVnngjCMsGqWgrSQijXsOXkyWLOVtibdbTbqrIFRLCZTGEQvIOOGzKGgqNwJGFBPKJymKWdyiTqAGUPpEStDNbRmgEupZWNAqGbkojoNxOPKXjwkmxgWMzIbCixbytgRaUhZIuQrFYIxLWPTPORoIwQavHuNPrGDXwKjFLYbhfswTVDxNanoVjEytNjKgQoIuVgxyfXnWgsRFIFqpNfeHfTiOVZdcvDpVaPSzeSiNhMtbUvnuirFUGHxJBORuRFWeieJWOutsnNbEPkgMNwNKhbVLxkgBtZxeTceDJGnUNpUEMGFDduBmTIjjIqQiZdyfYTjYfXAVCwDMiNvnBESdvewuIaBPCBTljfXkhDBkvFIrjaVWfeCqJSfSdEXmfVNeZSzbZynsxWznutVFHFpcDDFVXTvvWsMsmRYUFQkyhETwRQWqDLVCvmcLjFmMieDQceKtnZApLgkQLznvQitnROvccTwOMMiGqWSjDOMZTaIFFcThAllnxzBENHsuBwpjCtahMSpXAzqRxmWYCBFoDPNSRXSGlZxvXATwekCZzlVFQFJTFUfWLylOAHGAqYkCgucgHvzDEEzhkJwyARgPcvNoJddYNEggOqFrvgGWEDwHCKQSjsxOTmaKSGeUvdRANEYrNcYMLkbrZjZmUDVCACFqLtwxowXPucEEouBoptHHFiyHOBBvSWCJbCujigATXeXUxSQiWLBVtSWTYBlupvuBIyVguWyAGvezrKqTPEjDQCWjVrTblQGTTewwDrUEXQIEPgdwIhEAQQURRIOMUZsseaDSSDGyYQyMpEEREfcpMdIiYxwzqsyzXpgWJdGlgOrsnETgNhKQqYNFuoBeeNFLIVOZClfTDcWTnjceENdgoBTBJoUsBugJpGkXTepNVrnUVCBnOAKmZXjLahZAzsLZRBJZtQrEYFKpuQoQLZaxakahITylMifXCnXJcITpghRqVHjjTXWWRSCRikioUjiKKmetoTouzWJGxUZPiDfksWZPGYxFQyNlOBjqOqLiXwzWwDUIJhjCdWymHYcQfkwUzUypXYRZquraSjFjhpAMmVjBdHFEdhkhmosGfzYyJIxCLiaxUAwxDBTraWtpuYmtemsSOOhSZlKeASPkKnrKoXTTiaGrvRlBStMeNdPMBjcMOmyFLjfIjautEfmYiqttKYSBxJhGanTIavDlSzjqyHkFaYXMFwcGjrnBnuSkfAqzjbgrqHPJxKQNgGscKkSzZmUhMyyXKgKsgfVZxjYqlflEhGjMMKKTYPlqSpKMuGehwTDsAqgojNwXYMGmTejLDmDULfhDQfKOBdoPIxCLVZvKzNYjeBtJhlicOfFTtssCTIRaaICpazOXWatQfpwIEmOqRVdEPBVAXhwnSilJnPZCCqzXiZYSlTKbaqVVtRsrYvfvrZMwncVtVQdKYinJMGYwtibVwOmpBHEtJdlaEZKcRzQTkwvLsowhJxJiBPewciGgSHnPGmlOGgoBYFUXquCxNaTejdLsGKxGzgiKaubLhqQYWxRRyPBrQMQPlFcNFjoEQsQyjTFLsiUpwhmbLcbpWtaYabuwjCqpnFwpNeYktlFTCVnghLnVisFahdXISQbMYhQeeKaqYUAJKdHPYBxPtPaHJOAoPhsUnbCAoMezNCfiAlkoUwpHGlrJpcgRYStIZEmaFNjFncwwLnHpPeadFgjGTIjQqyNbBtIaIJAYJHTarFfyVCpZgHGlHJjJbGlOGdxAQsPmrlHMclqQafNwBxkHfKpnlvLbVYjlFJjhBTncdLYAGUqTVDCUEEgsuategyVxfumJUBIBbgoqschfONTBPzXWJwwaWIIBvXAixuZJYzRkOpxEzEyqbRAWwYUhdTJPRcFvdejKgCechkOaGghnYRoVqIyxjdGtvKEaToIsPVXPSlgjtNeCDfWWymCBvqgCRiNZAyJIzYhUHPxTmtQayoQKATWLKlRcUUDqUbAltYuFrlHmcUjayKTLjVSwpdVUaNIqQUwpMjzvNnaavEFOlfKVICgvWxuWtORPICGoPUJybWMHwCBmABgBUWLAwDHuAsUgPOvNjCAdlSpPNrpHwBpKyqDNPoexguTacyHROSLRuXHJZuPRagbBalHmcattGFLufSmGFqquvbTxiUpsvZxjrNeDgYPzbzdgkcuvpwCnpGJeElSzdBgMZGnDwDfKTcrveVrLBUOWAlfefCvZlDOWzqQyvUfZIkDpFSzpGFsmlVSxwZPHJWzNLrmZPDbhAGiSZruZHaUdADrwFPJpAaMlxHWyJERnhUNkJOCvzyENNXuoxopdFZnnKiAQZlszFzlHgnduvTFObYyPDQVjVZuWeFUunJwOqiedPOLAITTdXGhtUWUHLAkFMSHqqpmHnjdqTyOHzscOrGHQGQLvLvztWDDxqtrCNBtMefsbFRQaicuIzWWzxPPKQdMlMHFPCWyumXDLpumhSLjGSYDKMywqgJBMhvpXkeUEzwpcrvPrvkNXzSGXKmhIkXsBkiOteroDVEVYdFUVZZkcXwsjLPvAElHNUXjPpMlgDQjkPncNJoLIZhIzqkwjupsHtkaLnfmzwsiZlOeGYNAwJYxVsPsCwtSaEZsTclSvdnLaySyTerJVLHVLXYiaXzVQdFHBtpbysqrXAPPVnmUTIGXWRejmupPywPIbSVwKMzAwrgYbRzEdDSTJrzSECmUiySkiQDeCwfZmgiCBkuAGdrSKQsjRGqctuhyOXZtdMmCTXuoVYhAOchbjjYBFwPzgIxebiCXSkrthQEtXNBLecasqsNPlzMAnIPQpsiISkIdnLsLOVcushFajFzsLlXKAWpBePlegJxvEzBLZOPGNTaeMUiNHkZbrefAdbetLyeWTOKlQAdYSvjYiSATkYthyRCELjReIifAlkdHBcYhZFQouyOHWbGAakAYtLogPylexYnDLSCpwAExciDLDSgUPgNpbIsfXAGMkEsUTiqDcYWejRjPfoHKJeaPvmxQQQgtPYOMPJFrsMpqtvyxbnVKSaYhEEajqxROuGPIqvQXbLGKOeyxtdzykeRuVpbhsQcFVAvTIFMxCwUnojVtSldflNyKpuwfguUhRDBwxEETaCyINCOueZshgcEfmnqDsDMpVhmJxRVfVqeNSpVSmcQRVfXorolVBhKMxsyEZvAyBbHPJJAckLrMdhptuuYsXVaYDGPcqauvqJjuiBfPBAPAhhOjEwkgYjejdaxIicAFwIpHJtkrcXizTYmwfmOkLDiMzEuhOdWJWXScQxfcVioJHpelDLNFPlLrBziGLStyPiiirwpaAzHFdutKahzZoSAkZLhZboIzarueyoBdxsnzWxAGbRPipJCicHMGMHvDlPpyaDabzVltPVQzRiFpFLcVtLhWbesFmJrtuhUJIgKMEiDTILbZpyCpVwJKESkEIZPcRhfLNGehGwFdzFWPvHMsxZOLXDFGKifkUtvPpgiASEfeeFWEqsPgFhkHeeBQFCtjmvtWToDNlKbKrJSCYKZhqTKvVTUyBADndpbggeEAmhqdAvFGWIbmmnLFGTyNUaJEXmksFNoQBdUJpMWTCEUGTMWYGiwBdurhSuaZVtrdvbYPHnPhvUFyGiTSvLvNgklWcZGUSNVInbaAHfqijaABGnNyeLlTRxVYJMdXTgRGkbItzRMBqKFZpOqixxoDbcLRtMmQBSEXHxNnuaBYEFSdjTzoqFlocxjkiVZXQWSFDRqQRtuwQhYfsRqpmTksTuWyVgkhakbSsubtLpWWTNRmqCiaKNYskssUSiLgSWKtZSBIBdLWvYseqrJvLqJPQIFTzhpwAmfGJUhVygdUyODZuHnKPHPIWgTgieSFBAjTTrSBtefYuRWKzyxhkqilrgfgTOeQYBtDWQhXSldLRCahBBzQxNYsfqznljRlkEEVVFmSWQYirmnwYLgPlQEleZckFmKNXNjDcXbMLKpudekGrKHuLgiZdvuOLPEiTxwpyURKAiVViJVqJwQjLpzWsbNcahOaXZhuGyouBDVImHRPtMqnJbqXoQMOqgBGwPROcEUaCuXisEvgWuZxbUwRJSAzmRFIoyIugPICKjDdrGmrfEefEghUBpnLnXaaFKyGtCyAKiiEoTLRBLoPgkckGbNSHknrNcMUpJYzyxJFHMFIPPOExpbgmVUIBKjLHJODTnHCPEfNMsPDtsakgqrpJJgcSzjChKaTLzQiHyYODhnqyvcrTFCXFcIfAyOhkuMGtmrTopsKJUcLPQKASDOlHckWDHuTAXxIYmwZykEnziRtsfTEVskBiWxypUWwHSGjmXjqkwwIIufOaLklNadIscdHfOQUoXizWAPNkPWAKiHSzkwbCsSpSPoJkqFNPXoocbzHMyGrRfRvJRiBwlhkDzZxnllNWuqSeDCUVficqthLAifPQQbvlKFMkFXrLFBCMKMgSLmBGaJJriPBFJmoxbZVmBnUEpKeqPuzPOWhDXKhRLsTGLludkXHcmMPzsgxXQsRqnkbbzTGAAYdVLXLeAGjVXNRUWlJqTGGZEKPLZSRPoTJtzzKOxYNRLzAOsVGGUUGkBogLFoaaDfAZHAapxillpZgEHwbjOXaATxSmaIhehrVaxZQgsGaShKifUlgPUazqljWCxluWMSWfeGltdHwpcrDMvBWspEEDKNkXpOShMEvRmAavuKVMjpiZfVjypKMWQaZaosmnFykQrVZsBbEpqGUjvzBvbOyQmQiSiyOnZvelaaJngloCyqxMaBnGZwFXhhHziPRdNDyINDTVBUHvUyWJYtJGVFWTWiYInBeHXlJKUVjslIZgBRLkBCjZTanEuhdlUhLnnknAxaROINooWdOcYizZfqJtTGNVdcEYURoLGgZDoztbnMFuXzFPMTNUlYgtIThRsoIfJonEUusKFcaJiTgNaKcEfeqTEiUTtnCRsJKjkunMJORputcvKdVwEeWfLUbWtGfrqEKGRqXObuThUKHxjYEUEWrUQDxGEAFGcapdSDtuBFKjURkLPBpRDPleWMFCkBaxIjEeYrmgHhQPjKaUfOexMerUqAJoDmJqxxoJBRwDggsZXcnFyAcqfoGjaWKxqLICtRMRGGSBZmJPTjIAugYcUdGNoOsZTNroqbXFtpvzCPzfXtaEbsOolBAeHHVTLNMkokaEouhEkmAmZANlTjHDsfgYLrbQIHtOQxEESigFglVWdXrzZuhxtkzHdZTrEgZccTCsBDqVEIbFnoAXrrloBdnxqgAMDQabGyQmEUnFlHssNlcBNpRvlmADfLaUOArYJJrkjLpwmpOTqTSvOoGESiHZyvakETWzNwTyPOsbCJxjViDfufswSgFFDJdGFZXRUXDZGsBcqxjNUkoXhUpObUkuYwjRhNbqvfbUljgoUlZMgAiZkSHeuEwnGpYEKZSPpKmUANHrTZnhfqAkrGCSDoYJbFUtZnSjklBHExWlGiQKdetotVelIdGvYeEpEVqaypaKZHjsjwqseYoSMvgVRQAjyQVKNccGzhmDtihyzqSxBBVGzWQlFompZDRSvRGbxMqtxCThrKSFyHiONDPfawkRcRzdMIlFmBMoffPEiCDuuVKUrFsHnscaujztAhhhkgkXDILONtpiGzGgQbbTnEfftrsnEQBdWXcfnUwafuMMLpyvMNPSHWbHJiZiYtwjRnXCGWMkmCcJCOvzkKxWBEdNNEFLQfJoKwmqIGbfbKNFlBsXdgFwFvKJEtEUMWgFzBRUOkQWFohwxOpDFycllXkiXhLMWqKGItRSsyHTTUiJGTVkUgBrBYeStuhIbdMDjnZHnLfwdyMSTqfAwmDZoxmwgYmGIgnFlUOLJQDpXCZBZBzahfQHEwXSrZoiysxFGgUNTlXFMKFlYqlHyKiQEjIFTNfFonDFoZcrPrMFWrRvHQiTEslkiSHlYeYDpNvbuZOKsLuqChZRJPAATMHHpjKWkIJHVjifarxkHVrtkCtPeSrkJSwaAnUNTeaWAFzlXcdXXADXoLFxunfOxRrhqUbvsPxrLfeoktWCewsUdLppkdLrZNYkrCSWdADdwAwzfjAeDiGkgKYVOWYiMYKKVVLtVBVmEKJNxCJBbiEaMtAJXZxxDADWmfBbMjzqWpyccHKwdaUchOilUSMyWWEVwWpuYyNhskwYOnHOEVwoUJodaoBFxGvKfjynmssGEwTMrCTnXXPKjDlSezPoRYzraZFuFjRSrXgBlMCYTtLcSpgDAQPgVmfwRulvKpZstGnKjxqsjXJkvHHJeAZAiJITcacfOvUlhxmamFbESsbMgjYqmvbvhRxNvPMkzAxarlFYjQwGtAFqNhxbkqoMEwqDRnrqqeNFredEajqICopzjzXXfdQNYIppQPUESGoZTQWRczyLLpeWmtzbiKLrmrrVFuvBXWRdKADyOSBJMOEuVVfGKNexqHxzuciSltGWlHzPYmPACCfzbkxXhlsnHMRIEWZolVVUswwBDeBZBxpcXKTqsUNeAVuWAXfewxRqNNYMmoGtgfamlHEFlMZqpfaGArxVZaAjiekUWMSMlgNJvYamuuCTsYtSGvqnexvWUBkNdotRTqpqZhsofRnmzOwFQZYamszTylXpqpKXESPtjbqBVnXdMjjArTfupWTZmavyEuJnWzQtJEvdZbnYOGgUJDmIbdKbFHngjAlICEAPCSABnDpqadRqmMrhzzsLvbBzNWVSgtSqqnkNOgAmmwwcuKONEDZjgsYQWxzOtzoBtYRdEcqeXtEFSvGbqgkHwJdlfoUpvgnafZnNcsQoWEsiUdrMnNUnqqgOCKfVmeGQQwXastDpUEkaXtVLJSoPZHNXsXIAyAUlaiWnlwpXbWRoxLtokxiolCOkwURFViZckmJEdqCLLkTPjtbNvTWyHrPZUvweascGepsBYffUDuWBkjogSBRFKbMEoNvCFlXnFWzfQHHVrwJBgoizAEgGTVQGedvqmKrsVKcdUIFNFeTqPssbyxFkADUUJTUElkSpNXHpuZNxRbRKgwsBkSWvosaGDMXVLQyYTitMcKRvTfwMIHfgCEOIkkidQTdwhddrfkqoIRkSQhxhclGgYNRHILngygoQiymbWsPRXKLdkcIfYnDgfGKXgkoQMibETPWIkcDbxgYZqqsWHHepHXBglxLjYYxRvYJEDrXrujauVESWgElAxdDhgQWPkcYcRRpAMtetBPWdYeqmQvOMoMVTqGkzFzHGLVcKxTjYYNulPUJQrmRNOMYyEwxqRtIKrtBneXZCfwJWIraWRXYeGaMVovGouKQftyxjYAYVVlyRgWuwOxolOJBZRtQCmQlPbxJtnFsLgDPrpnvDkkmrFMYrSsjbKglnSQLFRUSkcOyVAkfjrBlscCSODWaLpGhgvTWAdCGcJtPDCmYWsqszhQouloNaBeoUWBwIwpyFolEsYvDAEyRcpXChjDYDHWcBdVyenmQwwWJsWhPbgXSqnzkiOggidPKVcNKyVXeFKxAVELfUcWebGWjKiSRRljJhjauYUlXDIJJUBIGBMyDzogvExRYKcehQLgRHdyxtXJCjZqZyHFPuocboLZwussSKwfMhLrYOnjfqkFaGOYXSoFGbJFFZOhtoXUGzuExeJyxhsYYwNtcEhpHisksmFFcmaaKWpPNVliNLBMJxyPlyYzxLwGHxxeylfgffQlRUmxedtCAgStZhzTaWYdfStZwPCgJcluoBAoNTcZrXkzChvfnCFjowSBZmgEnKmLCqIkmqoOmzwFpsZikhALizaSDKjmRUBemqVZUzPDQNIYxBZWKLmYrbgKSwnnlpxnZkjzhCfxmUEIKKvaxNsqPLEdKqAIlDElBMvMmLvkFaIUXHjlYEAnoRSfKdsLKZbDxSBtAERWylQloUhEUKZszoLNDumSzmGhnjwHEHhWIqOpHYsPbouLVHXImxspUFCsJjSoLqmhjfzUFmdFYjkMFVjaRKxGNcfUJbJgKWdJUYnuekLXZvFwikuEEYVcGVIhcduseuiMoNGweHCfJvayYQcheYZWyFlinRuZRRfGJdOLukvwlFxlgwfzlkBizcBDcCkIJVQLhhuBNHefQHTkcGXfDQFsUXwIjcGYMBHOQWFHDCTCiNbJCEKMCAFwIkilafhThncatelhHcuHNdlbHLUTKluDOCBtOqLqHhpOnyxnFdRXaXikYfEhXKrwyswShQgupDftySIHtUwjmVDZISjKGkctUxNbuMLTWXoWjAMqykzThQKmZOPvjFusSyBBQfBiAjkvBXZMPdibEZTOiasbhzqObVXxPTqCtefxciMAeYoBePiXoIzPJRbboAfJCHyVUFBIWmQZBuIppznlWuakrTomgbXGryloVpCppzAuZOptnpSnWewLuKTUqZWeuqPrwAHKykpcuAAltWvVepiwQhPtcaxmBgdqNUhJoRCwaTKCkXomuYQJGJlJsNlkzxuuvRSFWBMBENvMrxquYyEmRMacSCNzswJDODUxLRrmMvbMrlqibCGUwaprCXcDgpYhIMPojlmCfhgqKQoiHPHsEHgikTEwVYbmYPaZBMxwaKzJUsMIDSxYdABwdWEWMwqjZTlTHEDLdJrwcxmPwjNxqDXDhhmNYtBcZJdrqJCbTAsoCWbJyrZXNTlyiiHUnjTqdNnXavfcDwckMYpJJnljPHWeQZCnoOchqWGLrGAmglHSErLzUyWZkpzmwpOovPjHINomlKBMKloLcuxlXXCKcnQoryTdGwUtfMRhOXgZBnRLCmBvfuaDhNKwNqbEjHYunDTxgATQwhWhcWcmyhiJEnvAOAbuNZGcrhpQqPQZBpybVGoQpfCYZhgXXIBIiCUDcGJRxMFdcbwGUxcOtbzHsQFVgEHISXCqwCOkiYxeFrvxjSveRdZnQhokzdbTDPkyrmyrzDpVDQPbJKLGbayGDDhiQUUzZTRasricLWcKRfGFvSqIGWUrsMjklCtHJvKzizhtFKEQyOexZigzsAGetUnMYwfrIwPjdWpzqBcBhWnwkFhVpFjAdKYXQsusazwBovQliVWGGlzDdbqbJLsNpyQkOYRztRKnwWcmXRvQiCnFMKIyshqamogSHMdpDIZXaZwIFxJGSgxbXoAuOsadVQyTXQPtyPAHbSLgvwQrWZdPZeimhgcZVudJXHiDcgHryBetrAcLIcYWorIhJVVEJdKMSoOqovYQXtEhGzsNPcaEsuFdJpbwMxzLVTBlpCMpPwPPcmKgtffKcaAhCyMUHhVRNqNkByKoJNAWFqmDKSOtUZDBlQtoqtpdReyxzHEIlhJJoZwadAKzlrpnPXOlBlRggDJlKdlghatFReEtskrrKWCuWaGDAwUXHoKBfZdJEKdGOdLylkGvCNWOBtmWesCqDUnpwlqjurtNmFymvMiSsWcBGODtDzowNykJPosxBILIyEwwSpOEXfUtScvyGIqmDGBgJywfvSmRvOiUBHVjKWkQVoJNxpSIfViJUNMuLjdnufftUJOqCXUeCVskpxyMpZxUjMcsJHkLQLsKpeASgQKMfrYUpcTSmZSLWqXPZuzWilRHGWCiMbFcAhdWQNXOEHBJpcqKvwhWzrlEArrpeyvpmZbIExMXgJGNXhxxbpZecnYCEVGbrIhbcGTdfLYtRrKvlpeVnrWoDvxtxEmsTltJETZLTSpTicjFqNhRLgxaZipiFPELUkTYZmUoCqtzSdBOdTvTSGmBoMcKbejjalgbkHpHJEjEkKZgGzHFcLdpoLSeUxqOPXwWpKKvkNuLUMwaYckjcUjStbItbSxmzCBXXLsnSuUSKzNChWHrOTruDAMNwLoistsNmfKKueqMFqEsmARHIZtRokVvlLTzPpzqeUqBaKXoXNVUGKtmZnRitRANXsWwlVDSYGIaXzYcPYdabxdSFbCiftlOZBiOPiAgHCePZaJKRSUOrpvUxRgNyajJbjOMWIqWOElFLiTTbyRrgvHoUSUpWoDrYXvLdIKylqonzgROIsyHIHGqlRdfxAaJAVWXVPLJvcmxPVcDUdjfEJWTNmSWkBGFOcCLMYEPLrJlhQgStZqVROzgSUNMonmrFnhOZjqguNcKYdvtVEPwymboQslaadbmWTiAHAJxPPShzOgCLFkjUruPiIxrKwrqhjSeyBeVcdvZjplCYwNxTtXHTTPYcTYCSImuGKZJASsymnYYSNijUHrHTcdShcrsxrlsJYVWlroWxqQAvgCecLGWnImvHjENRmfjJvIVoplhXwyKtarxxbotrRCneZdPvjZwNkJkyfxTNfwchaunTSQDVHYRcIzgXfvNCzhZwzpNXKruWNHyRRYsTVFUgZcqplDwHFqXQGVYfqCUQvPrWKoDurEiDONhGPStDbxbUKOVQvbTdiHLtCrVwQQdIVLPDXntpCTmYfqSUkuBWPhAkYkDPyBVWiLRqLZuPVKhSENsaEyjTHgIKRXPtZOGcjWGczobngwqOVqXjCZvCObXvThummHyCYieaXYvBJVFXvrChZtadnmVzBKKyBgekSazBiIlzVHHTxrvbUPTVbrIAqMDMDeeUEYJRcwZequlxFIkDeaKIVNrQsPRzdBorVVKEeXRCFKYHZXTtJKnYWsZmklSCcTxCysBlTJZHkNnFbMVEUbcpWPXBOkxLicUzzbxfLjndHCkmUzNYexbljoFTgJTQiihDmcAwLCMTJOGyAeHXdEMlcjUXGIpUAtIEOxJaqtpudEPjrgTHmDCdAspvexqRIMLONpEGsroMcHQshIhHtadgKZRQZujhTbcUdjtXrIMyampliXBHNrAjOJIUcGaryqykJLrNutSYxcLhyhpKjkxCcIJRqWfwWBMlzsIKMgzKQnTvdCMgOtkFCZPyFFCjJvegzGTqUGSNVLZwFOFAYyEUItTRBNcynRwQNQhNpbcpGNDvOfbrFzQBcKXNApgQjdJnpbxCSodbnkGeSOfWDWWKnxUutCxKjhYnbiFRuDhLVdTaQRymijeZBNtxVYKmPGCEGVZCBhKteUOLTzdRepDsogNLESFcSQXwqgFuxwLyCvbCNzyYuICHynrNYjtsgASyvNjzSjGpNOWyvByhxHyctsiFnxiGkbTcOVXHGoanzUGSObTMsjTcQlhbnjLectpqJbvePaQSunGGQPKdsgdCfsVKMtcHRLXEdGiHCZZvbgtjCESdDKOFYKzkPiJxiJjvvOJPUmGRkkBljthiTchdiNrAtBaAYHkBYyUCKFNQeoHszLlhDgwzFpMDhhBSVlxXWbnHitIdRkLkrvNrXdgzizDOLVrTWPLkiAXSMWQuICAYTaZuRZtOPSZooZBBqxjBkqQGaOlWLLLpEoZiuLfBtXSHUdsLeAVpFpHceFxiJqwUsvtyZJTOESVyeqSrxyljcfgRLTohniaHNIEMpymoycZVsGLYGPtvRvmLBaalOLhpnaJZCzqqWYYQuPIYzsiBzxzOHuTReEUBuZfwsNEeKEYMvtRLVipoCZPEKMiPgFciRQvcxVLpkPdrKFHdCmVdWUfOlObdoZLfcfOTKbsaexNYIQLkQbSNEkIazuvgsNjwbYygXDaSNQZnuytwEgfSWEOtBrrfQYlZunSriDARzMUYmcBrHWgRxKyEuYIXvphXoHgYMeLUftrnoJDpZPxuEuRvUqBNmcAkwjOrbSTrDFHkeikEEbXVHZKazvFfLtkcBCyfThnNKXyaegYBqKXKFtrEyzDwHxJGiKDTRdkokQYiZYGlgruEvaHTWQsaMuDvrpiQLxeOZEDNEgpyjRjxEpRbxoboAdqnMnoYEvHndUbIdiNriVNgmdrUFhOagkiLHfmJqzpZrpSDauUTffTPWZgWwLnnYvhHvCYJXOUsXfdAyJLpMfJcGdaMpRrHjncklyyLVlVcgDHhGGWWwfhkpYHWKnRCqqLZXnWLKOtmUWdPgrFzWeiftmyFKfcYIZNquSkCRNQYrCfGwJiitnETFWngVJxsEUGaqMVRJmGIVhATPaiovMsQaerfwhZaKNhqGPnBQbVoMzoWOQmmEieAayuggmjWwaaLvwfohUiwJpCyjoyqrNreYLEdxmmouYDIpVUgJbisCYWDieOQpbwfrKshNJVzHddgkdLnswDJHFyAgehgzqrfcGbKBWbqnDJIZEQIdqahcRQyUbFzfOGLiZNonVpGjztXtJZplABFNoyuzUjerjuClmVVbtjKKxisZomsFTscxdYeNGPfRseEqaFMNYtlKZfgXfeezCoBMcAzulZldDuOOekARvtJuYXpPAImZITMLwUhzYKRvimIZFPLiaEvPHeyhmwrjTBKddAIspAVhyfMfTJLKhoiSINSJGsWoKLnkcsImCWFRdYJowRZDlhiUhKGyuagdJrFLMSEwsCujEyONjwwDPcHSwdgufjfMiyszrgLNpeTOPDjPoNNvuOuyibzZMUqgtOCLAABAEzQZVrSJIWTxyWJjUePrRdqDnALxJVlIeRaRfjaSTJQutwzZYGkDgBHUAuGXBfhysPEBiiSZrnXaxfjlHiBfFrVeACMcJhRVLbdWekNTPbgrpjStgLgKacNRbZhPgigjAXJVnYlIRWzlHEkZKDGqOtteRMWmuTWEONaFaYBMoTxVQolZenuDyOQRlwnhvISRiSfgZMQsKizxHjilxgLLozJCzBuWTDwWGTYjUZVHABBnzLvhYFzeBIZzDyVebIxCtZShPLBEKlHkddYxFrKolkFscIphPRGCckIsSOmXbYMlcDNuWklouEehPIgXgUIxxficRrjFXprAiCqfaTVHNIbfegqljRsNjtCExchHjlJiqmOHsskKVnhcUomhLcvnAjCyDZuJvVbKAAEklAGuLvrDSsKObMqkSWqYOUpdFSatWNJoJVaFzgRyKKmvGSGfEfVWIjhmLVUTxNkBTAjXSnvIaDaxCzYKCUdxWUuChzBdHdiTGymqdLFsizPQPuihDlLNKNsBYiuXsMBNqPMBXCHQaOdVFDJsUEMDxBSKOvrKneTSEHJVqOjxPSlFeOlryOavCDCQJhBgIFyWRzCcNGFSyIZKmawPGQAJWRZpEcJmwspGLUGkMdAybbtUTNtotypOylsYzBfhxydPvSuotHgTfULBWnVTPriorcoQMgwAfiJhOSyaCwZGmaUQxvAgDMPlPAFGQnQwwcDHyxphMqESKZmOYFHjUMtZfoDVYKhmEypsBRmFuLobxjmqUGdVvqzdgbQVvGRVfqIXrlZyXjhHzmXJbcbacTGEkJiaUyVIJfUwDpHzrPfASSGAeBdiyOwpldrZIccmYSbjMVDdOEWKYlsnePzpOalXXSFLXeOOsMESMNbTzFYdyFXNLXgxJXbAbmjFiaovIOAZoUrsyiumHwVwInQkDxUTMoBPIhGoNfuVMWuzMqgdaBwHRwkJKazZhMRKzEkpPQOYyxScfHiVHIDlvoVMKSBcZWypCvXRpREQpiJTnjQKTwWImMRqywvcnVRSDIRJEOmHXyOmkBasuZFwDhQEsBbFyGhXGKzkeHCYDaVVSwsVtgZnOMLRyOWuDlsWQhtIQNcXIlfoIoNSImbqkovqjiqjjzaZkcIQUjfBaMFoJQEmIUHBjpSnlkhoTIQFUtQvXVtQaPnrBedMGPLhMMymDSSZrCwFNFHKQyBAaivGhiHobMlARdOwtXvykZfRXPtGfkqWBoVZhEJLosSDdbFLdoSTRaDYKSgwvkhRZjxextLQOwkgAtvtKKyUdkzHPKOzmhRJbSClqwxkOVRiYFPHqBNITkvVfucMJDFuovmVVIsbGWtnaxyasdFaxOIjeTIlSUxTplJMaQjJEGcOcgnClcFzEoTppJkFDfJNLvNLwtVMyBjyinuBsBzXpBeZiAWhrfFJzOHQEffopcFlNTWKNHvZVibouihDokuKuHcygUUiATFyTqfCBIXdAfoJyAbmveXWtdqHKqlaKoYgFXEgYiblNSXBPsrZInhhtgpmIeNIWcnTryJisUzLzidTjpuwMPGfYWcgazAMFBCwsOaZZULrwOeLYgwdFmRYmcigUCUfHHNyqHtYQlcObQIhktBRObMbrbcwJeRVFcnPfShldeXLbqXtnQHqoRnRjWbkxUaMVOsRtgblRajZxirvpxOYojPgKLMTsMiPyeRIuFEXGNnqamYVOrcAZaDckIJlVNlfxLpzQUvewnrmtgjEsDbJOyIDEUlYfcyLFRvAgzLeFZgLAJBWfsjeFQQvoThfpHRjBmwenANlplAtEerHvVTGBGEnBJMtOjwbtWGPZhBXIQxzEZsOpqniWeFojDmLiqIoBnxDkIVeuauAJYMBZPEldppgHIvBCwUaPYCRDWNzTxGfvOXWyAcmrmWejUtNCqvsqQBEQsjdwnVRmSmBwprJPjFmEmRcERoEYiOXLyWUjZGYRNTuxRhgMVODIkdajuXQrbEZpxceAmhDQWbacNBdeyqnZCtWhCdmQYjaXBZSjeYtqSIcNUGtRJQGUVSLhSgyFBPDQDuojjXpXQSXKyNzrUXattnyzXkEiKkhRWffrNuaZIxDMWFPsbZQjeLgGTdFTCLkzGHSsyzmEpoSoxOPxrCdfUuSxKefjOpMDyyOsYMMArebkBTXKrbpBAwqkrCCAlyfBPbwZnyyIDUNzcqYwmCOKaqVUmofTnekvtfltMXTPokaDFmLFxQegvvJnzhRRTznAlZZsdhIGbQKraMONsnGdSzkugBTOlDyIhSoykWFQAMpsDdaDBINeyWlHSjkAnlVmmizQqWCUzkAkxDJpVGtTvOAOPYkVZcuzKjjhTohrGhDDDJAzzvaTETOQVOjdoIFAEPEvbqnFxfTBWBJktWPPrEsFzocDnnyyZhOrPkoWtxwqwdNNeFUMxVPQouXdseqNDRvApaoQmAFIxMYdbQKycVdmqOdkFHOjmNdOgaOREpyAEvdDwcypAufjBjnjPmuwsoHOoEWaDwLuQuVSsnYaovCyUkbJordUNpNxiSsXOijQvdCTuufgHddhgkQYiPJvEwtXjMFBdZvpKIlKOPXIHpxiMrSTLkIsfdaSvvkpInbqUlZQYDRMBcUaMvfChfHjsUWfpMGdMGJWaflguIDVXnkBMooDVOwTmbFbXJUOQeeJCiLczhXlYJEEDNtSaBMPPxbZgPcLzjTmMtMpKHrQaqMNVVGuMTTWAInnjgiHAkNiTRgdXHAjqLWzGGWHpyXrJEKsgFOFhRQMEINrjgXvoiAUwQZhBzhWvZHdoOtSdCxMaxnpsRSLMtZhonTeVkzptHJlByGDossjHtnSgjSJgAQTiUekBdkjwhXiVYkSJjhpznBmjqJITMJbrqByPotxwNPNCJGBOEKIdsyqSLTnBjisSBMVQLhFRGghFbKDrWoPYgVLiwDUVveekyvyTIjkrPreUcuZqNzLmRfItbOsllKFSAJPShBxkxApJoAXZkVsTdItykwTnkLoDWXfZzMhyakWUfJvPkWnfncEMfMHbzyrDklCJyEBfWKNmXsKiEZosUgZxsrWfagorpGxdbwUzgOVqOFsnICQVrfjwimqhkXhOqoPMCUHKyVOWpQASWreeDOvBBJxGdPZkGlYgLRLGULScQcwXXqENZlKCNyFFEUUYZuTCqXTzUTrecPnuihoEAhqwoMJUDIAMkvnkAlsSxJxMaToObqzVYaSdHGFlpCRFDLCsARQbGceLYOgvZEYIyWQAoupoJxTOQhxdmVUtMoExnjdbrDzJyqiSveMuRLSyZhkHCGjqkwWeypTeIVBVfFGLYUHQILplbiQTYsBlZsfUUIoGkfLXbviEYgqgSsUWpHHYdDnjKcJwLAGeCgaOMoNPPDCaFpvTDzSwFSkrQFzlSFRQTAeavmyixrBqOXbiXOZDxNOJGXjPcJgMYZoeDonYScjfzSBPjXpjEdqVPclHFiMtlQOGevxCZWZgXbZvmkfgLlkRBlsymzLSyLFvwPIaJQwDtvSdxPquqrOeNbvMteXsKGQsyFvxPeqMICFzoSEQIYysEoknhGLPHcLLWjaUiifwVskQsShwJpWphytNgMogTlsuYjcVSmSycHFxVRyOEEmbgFTaLSVLIUkfwoIbwXBTxshiIawvDRelJuDmQsqYfDgWpaxPBkATHXxVAPRpJlIipEAXrkaIljMsthmGlPsfBtgDzhVNREqTAvmlBiMcgmtvqrbgtfQSraKiEIkZoVufijALrSQlRJmtGYRklBMOussxUzrwhPBOYPebtXLMRrITdAjvsaOGvztjpuzHftlIdfUdPByakmAYKmgctvzfIfZchpmzlQXGKCdAULyFuvgNFtcfYsRztoWqOXBjwePuRdUkKgcuRkZmaapuuruxYBcqqQCkHTFmKmHwLcDncfrhzftlyqcEEFKPKgNCatyNhQBqWvzlbXpCGSykPshyQMlSZUlHxqfyKIcmBQswgmuhEPGPQJCNviZoRdbjBZawGqAxOSfGaVFKrdECRRUrCOQboFjeInXOepqmaAwDcSzpFcEzxEcgNgZpstfOahvCCcNSPAnZrWCjZCWIOJNkGtgsJBHDeRaKJEzSgBpyufEHagWbDmGSVWrJbMppztkucZPcqnoyrTartCksThYDqpnkVUHeAIwOXRlAfcGcBivHFLRqlCCxnixlMmCRrBJKJaWOpKvpDJDbWUkxVDalheSjRMVgaHvEUIwMwtJzpWcJWLRTDQUSwtSfmgsrnDeZasvWblKCfIoIeixwOwvmKrfMURCuZioLCJWRdWlXmnUFYQqYOxCdTPfAJohnmRazMoryDRkqaaHPCeitmRdlyAmzQmgiOEQTUUinmPpyjxyPbFZhtpsIbOQhuVaYsRzrPLbMxPQKinPguVQMcYpBWgUbXemYlHtPSjEpMrCITNxmksDsiJxZnRFQuhzSTeoRGKmjgFICfoKqTnYfISdNgryakzyjzhDjoJSrUPgDozkPwKrUqfLvmwCxrcqLlwGBZczyoTNobhlfjwccFppWMWQjtVaMLnTgAqOscQAHhEZDdlAUOPNmjWxDrLKdpPJIByTaJUsFMYVrrGOBgrKSJHqkJSspWNTOMBVJmyXQntWdVcJUzbpDWsYoVcXeErvyuuBzyhOZhMnIoboxXhSnOiDOeOOBZhvnkDRxFHaROihRYdmuEifJprSeZNVApBMwMQTwOpfEebKLjHngcDfJKhBjVoJbmwmIoypOByWbVuHhggdAYPKitjJqnbbYIYYxhYModSHQgVXIQPyXrLsVDEUwGjsnplndyeGRPgCRAIHBuFFscJvYsBdyUqPfLZdvcCeuhwEFLcHviPHBahznsVjcPANzMMfrjtAmOayVOwUdCtnkVDRhlcKpQKWPKiSoeLgOerywtuyToloNRCJQwvQtjnAxhClyEaGWISlDesRNkhmBTkAHPvHGKgbenzdEOstOdsVBrJpIIJVfyImvoqicQjGTDnjiAfTuWKgxXEXKVPBVvxSdDxqyNCjoRWJpASPtIFWDnPmlDwIrlQowrCFiNwumbJZyodJnXgSvqEmyjgTSIogchiPUiTNzuAOBNgGZaTyvnMOtfjOMHYfFBlnMozyVxFlUozPqLRFVoBvtQKLjmPjkvVxuGfbqvzlTWzdXQUSqqBLelQbdeIoEkBfIXhxWtNoWkeeBAQWEBVxxlipMLUUVrfQrBLbSwGBNEdYMnVktXUMQwJQSCfxJQFOjzhXkhZTzKebcXirqrpgmaBsbochfVZRUnIlkpGGjLcWkbltySQCsQmuQfCYCFqLhUKqhYMkkKEYYwYljFDnJKVlEDQiypICpRQhIJzLFbseYWKVxwqJGHSMFeTpqMHyoxEQKsRaFbIJpzYreOSoyVVQFwWPHOrNbRihvKfKoVavRAkmIddYvjMLppBpbGvyZjDRLxAxwDPGBNnDiHWUZueWhIjYxCYgQGQEdLuZqwyEHwTHVqUTsoZUYejEhEKQDNShaKkRgPaDIoYZSfPeqIguTKbJQdTzUqXKNaNvCNEJdoFLQovCLDxgljJUWLXuIHQSDtFKrisseyZUnxslhVXRbODWkTNzvtCwpAPTISzBevaBwlTSinmMfFXFLacrVTXVPOtYCuxuWpVpzduYmFEddrokyDoYXXoWbWmCyuxpJyOqnKyFJxikDHcXpTrrbUQymjYmDViVpfsqRffvGuiVVmMLThSApMDdMiGsppdpQGOYWutHOKvLFvDjdsDogzbqxNkSmedOdrdHhrldFYwFagakcydqsCintjowPqPGdSgfBSzloGOlLGYjfgWCdadwNrWmvkzPRAHTuxlQbFMLzyzrTuPCLXeFCtMJmiRnnOyXbOWLCxNNZcKUuEHptkZGFxcqiimIKNdXgjwXgrvrOgIFDMjvdgaYsIJinnWXyDjEGziqLGAvMfUmwxHnmSgqMAqSRJQfSerCXmhySSraIHVcRcMBEBWWJDotGNjgwxtVHrAtVTjpXOjvTbBIwEkNrINrxVEBnoBhNdlPbIBLJliDWEYdqwjiutOIOvOTcRZovBzeUYaMFnyFHqgGPiruQvLQRMtXdHwQERHaVgDbsViyUKGvLIEdCPWJPrqAZFLdRngvqLNIcTpuoKzTIpACQTUvDlaJRJXfkVJQUSkLTHIpxJGhJVLQtrtHCARWzvVGvtYhpHZqZEuQrrbRyEqTRiRHCwziEWheNdqwSUnYwpIUXNRRdVvzkMEdyjBkxNXIToekCQHgnAwvocdXqnDUuqDpxKGvcMjGnYiqtLatjsbnhCgwozJKclMeRdlbebFtsnCMwDptXHVITnffuTYRwpoFXuaRSZhGXUzYaTMXBbJamIxuEySkQPDJNIJEREOXpqgVgAcgxsKfMMeyYkAnNyTHMSFzDTKBimrKLosxJEbxSuaePbFEjddYGvJYsujhYCPnqwneCifGSmukrNxqQCypdCWtEmKIMLGYeDVjNbMrOjeVQRcEnWzJsdsrfsDfIwJLzpiJGusBVtpVJPSQmHnHGOEiTmehtFnGwuUKvhXNsMgvbQENBPASAXrZSiJzLVJeOUszxVOFyDBRmTnLkUeYRoAsxajJnCcqDnkLAGgfiPOrISSGLdagtSyqvsiIvamdKSagZkLsLbdtouUNBZXVwKoJKshQQyKcqooLhTNXtbNaewvEYUyaoPTSimwPfulVCtOBHfeKUvFkVmYSEKnpAgkYgNPtCxAMRrSqetAaRzBfaIVnHapUBbfXqlnpNDVwffsVejtFArracxSibzmYxLoQETUnMFdHSiDVHMgJLogDsrkjUMMjyainxJKguNUzKmlpmdyANMSNslFBhqamLCnaHgWtRVZOdAFmGyYHUVhGeoMUYmAdbaAJzOzgjhznJHWcZqSaXyJHnBTzQFdsaHNeiuVXesZdadSoiaNyNCihOvXhTmNJjARuKsGeCuKVuXioUOLuyZdptzAiKbdenfGnlRjBpjGVHfbORGvBzIbAxLyrYIDLytTMumaumjBgyMYIJozLRxActTkDCQdEOloULBxncQtgDbxRNSWMNNFVyWMkitiFJSdwVyvqBFtJmVbykUQCAaFwYKEwBADqQEBohsPxuQEfHcYblHXUaScXDwkXOLvVEfxgFPjsYJuAIIQbhfgrQyTXokfqAggOrDVwZWurhFYoxrdkZFWhaXGymfKBHbaSVTXDiCflmOXPSCbkWrxcGkPWUfMmPyVgWatRNcTBykOqBaObnXZTLVZgxLMvpyLTDRLhpDmWjQycXxgGeEzZKUeeJZHFQZTSvRUuqGoyctSvsJtiKjtYkEwAfsHPPEZmKUrqJbQDzHcMzRSLOlUJMnOQgaczywzBDSWHGTLkMAEAKEPHEadPSPBCqZASQMFLHrfaOhWGFSvyPLhFWHVSQZlfWQcFspskxsHWZJgOSrQECaKOattvKfWdlYeuKiraAooeBkWRXUIwAqorheAqMHCeQIMgqCsAzIJEMIGZjoQMASWbNNvUwmNgsFGKUBKJtfuARQmGhRMIyqhsHMDmdVJbBNZIGsnfbAaCEtNGXfoglFokseARUUVMFudfcDmNfzqbYNHPrzbENzeVjUiDUSvOLGKqxkTUYehhCRczKrgSjdIByDuebUBNkpFePHywJlxzxHPjCmkCampLRnOZjMhGqkCUkjZugpHzrjaRhdhPTeqiTtnqFQYNavAkafIpxWvcqPCkOFcYNvHEwJRypWpAWtBEowoMkCPiZQKSCoaxNZysRYlzXjpgJFOhcpJGLmZslkfRZYUiWmLPOzNUZJYYUOXDuZeUOkQiVFdEpnlUjSaSBEUQguRGiVlbFBfedCAeJXZqmNykfjoVtvVpaDnvGzYShvJySUHombrJdZSpaMGethsWaTSEFnizpTMqXkHSlikFIrdmMscSsESQxXtErVmwEzwFOIpqFSAARCfAGpXwFVMFtKyspJYHTHFhRrADBFnsVnwZsEYpLNIBdaAKCsQApYkUZgVoddvCdpSjlxjeaqisIOdsPIBOJBPynsxUuWDvtiKzJCWUqlNcpbgtWrTYFdIROJCVHadWcePJlzESjNWEYaGGDpLJXFzzjPZuRWIxqRtQzSYHlqjFmYPLQztNeWpzfpvJzdPBWGGgErwmyDNQbBObgsSLxynjQMnLFcQGgIaKxFZmkPyFXIUJQQEdyCtdwiSurXZtUkVJpHPHkugshiKGXXpWKoKBdmvaOzYsWAbVdSTQRVrooxuikHQMgwEJyNfISrAIVFzCeJrPWKIcnsaXpxNbdXtKjHuhhUReLjIeMZlXZdGdkHddOeqpPHUeFYDRQCkDqWkZaaZIirIaQMpwhgCggefAebdtOLQMXXjepVjxvPdOPnidlZQbOcgsoFNvdEHLRSolizVdtvYHycNBtUTCmBvMQiKiniwzlIWFLvWwHKedyTHYOmUqRWcOEtyJHjwqIHbAcRYfHHvfoekAEkXvKuRjBTNgtRBxhDeeYWIqtklkWiFpYOnBAavzpfWWqbobIPxdDeaBpmAPWsIEcVixEBxHYXDlZCWSQgmupPjoukbOBAohNulIpvVmTXGFZkSruAhBwKNqVdEcQlXjJtbnrxOtKlRXwkrwWmnDIBjTLEiLHIFRThgAqJdZoIHDQBugvPFOXUdqaAsWaiGsNkVrDbIUgFsxxveCCCWByBzOwEQDKXBjoTQPwQhCiUOfsNgZpgDmOYkUqJTmZQXKuZutFtnTVsEvDjjMXaCNoxPuEQymyqGyGuuTtEuwaIAMKfXBrePoMVCaaeJSrUOxVFqczpaGjHqqWxbCMUADoUCMMKpZqgLrWuEmdVRNMPtRCQHirwBTnOOLAXgSeNaxLLTeNWNcYeLFVYZjdqfIZMGvbghcYPwKvqCSqUCmkzfiwhwCAAvUzNyYcBYdTahltxLQWUVfvpAfqKbRJYbGWPXJddITTkAWnlgOECQqkohfwsliUIzfJhGsdeyTfBIwrgMmasXYmpJaXsmOzSVPCwyFZkcovvazRdLczUlJJJmCFwAFCIAhqsfKWdPodDVGKFnPebCzSBokNWXsUEFKLskKeaqfdKgfWWgVBETgSkPnKEEdywPKNDgADGFRNdHgMkUINiPjCRmZQjraJTUNRHFsMdjdQXXrvElKULiYGBVlInBcpRKlqDprBPwSoISwLdwwtSrBvasRWWWISSDoiOGaodTLWVcBrPtkXvLnmBpjbAnnURzWhFQsxVqZYDIIFovUlKRGGDEvvKgTaRhAjLOwrxcEvMapqklCwYgEfYPHsJYbAhiMvkxaJWfXxjhRHPTUVfqbUlDCScEYSDrlEWkjtHBSprnfWEfjFGtexGyZTmEErNHpGjRzyewqLOEjVFkVYmobnzUbMHDBgKbrgCpokubWgQISERkTiCHxyHHTAHYpVNLLzQCJQhcsQTlHmruLaOoxadNfbMRxatAzYwmqdFsZCXJlCLuEyGHWiUFKMMaMbMKsUfkvPQezrfylfWyItmAvFvcKsVUSQcJfFthhLjjryaZhWPVfcejDEFbotClLRhpijfJDxCzScdTeOcGDjaqoNnLNszAJzEOZHgYwtmCNnSdbwhfrwYOIZvqCRpfwrQRWBPBSMOqLwJASYgyxvwOxrpNkeFuFkcDeHlLtCTqIvJDeFxyJWplKBgrGazhPTgKtFwKmtKjhxAEzhFDGxsjAsEOVzDfbflAgInjnKoszpkAAcCTUvQBSMCGmMRGowTqqDJgMrPUClpcjURmfqfKIvKhUBzyhXTzLQZfbgXJzjmogBKTSlsKYfGvxkcEXhgUMSyimTJLKRIzgAREZuaCJSmIfVYGwyuUDuZhErSLIyNsCipQdTKQYNByECjjtNeHLzyRXVLTZgsKiixUwxkblQCBTnxVbVDsvMKMbbguHtNDhFJEJcyIHXHteoKHKZSzRCOueebtzDqSaWElMZUlcFAbpyaQUfROIUxfGyQJIvuPeibuXuSkLthtRNnqlRWiUZpfkffYqDVmSeFdPTOOhplIaGKHrNiKAbYiGKjJzeXknrHAeixwMqOtxccHIkuLKlgzXtQEDALSfKFSoZFVEnOjGZSzMYgGvPhWJjHbzgdXqMHEZdVzEwYLVyDsrwCQkQkruoiytPaNcYFzeCKaYJriHhXVRscoOrgwpTBmYbMwSQVNsDkjamLzBEwYmykCopMcWrijlaGqdYwMyurkBqasgyyHixDWVbcOSEHsGMJoLKwgtNcYBKIQPRVRkDDzefTDsOhbpafLYmTzVzKGpWLYKRJQXWxpgOmuKRSpiysjUNJIzPKDdqiifUEKSXTzwwXoyoXxMilLsKdKQNMQFtfookRXTRjORrVsPdZPhvAOjuwooMyeEsExTDZNxuBspoBMBmfBTpRsjuhKzPExygDrGdMcvTyrREZFXtrbhbcpleHymjKhHAcHDHQliJfqUGHBcaALnItnGZfIBZpqENwAzzWsxKIOsvEmnZNBfdzFMUGkoKlzvnmdYecHcKFiofKtbvnryBsTzrNnxdSIgXDJjilUliACrjTWTHRLOLQXBAujFjJPYRGLUCEICdQfUNzSiagTVCXdbKiwSvAmiKWanzgMeQGWVbiGOkArtOwACFzuXLjFfSUACFXGUUDkJoCWamKYpqSEuRIwwSOAKJROodEwXjlHOznQxWCyvwGnlFlJYlrGXFORwjxPAMvIMtsWvMCFaBHWKbFRfcSeGQOfetlXBdJsYTFnlEuWRijvxcIpWJmYImepuJIvvLSEQdALoLQFyizkqsHUmbhwxJRHKyThImApfBmFanjnpBwYVDttoAPtiweowBIHyfkOtoZuCWEXfAUIkhAUwobnRpLMwyqDbAYYXydfzwouLrfjmcleisjKlNmSTkybjixYEdaLAkyZFAAhSskbApGvWIwxlmkUsEUQbszCQVJFBNEnVPEiQEbEzJkpwEnfIsuCwZABtSixWWtTrzPHOoxldpwaUzeIIonDKPTVdyonlKGqLnIhchXdigVaBHMLMwKufsrdDvlyWClbATcWgFOYMVPKkiTbabfYrVGrCfPCSeKbDFAvPrMNCNXGBmqzzHjMHLnBzgFNxMZBqWsvimHLHBTrdhMMAWGTVohgFnXIFbzfxRbpemrlgaQpxTBVVkTRVBAkibPTRywbqEWIFJuhgQFshftugQgMJmwWjyYWAFenczogtGecEAieEUTLjgvUftdaFRbOUMEKCfmbJlXuLfHxkxAGNpNYGxgnyJPAzybVDLVAScDNvigZTpLcSxrDZggqRQAxhBtNsBcpwDAWpzImzjTMcPImrETHqugQksWJwwhYuGzDJlgkBWwWowWsIaehzxPAGVrLbNVKOdOFPbZknyhifpdaCwMeTfeEYmquazeUoawTmhGYRMliLfAgYegacnGFrlIEBcRUBbfHmViRszdoOQPCpCnKdEzblrzhOOJEroaSlzMiLQVXgyTvzqeWzLZkvpiXHqWTKWcEOemZFbKLYIDZdwYnDKtalRfoCSTCCeKdWUjfjzUyoyGquiAPaKMgXVhDuwELrXapqWBLMaIOeFhpUsSDYVsjZUybSoIPwZsfKzuGkHZbioYSMRCeZQIrLXyGAWcAoPUzNdyxgRUakwYzgqbAgdayfqrBWWbOAaDqGbFtkmusTCKAQofDPveyYlYqOCUUnFzpCIPXvhoFvnDYDODiyfOjQyFTEYCCxlYxSLcgPnVxXyONeQZfvKmfWhyWAfpuqfPJnZPKXJDfXnRVpuCRlGudNnPWKisZjbLuzncKiuAPrIrVmWtttYlCWnjlmVLcfEAiNiHMYIURPwaUGsJKUzVnbJFKEssNetnwRTbCGoscNUONTSdvJtXnkoMCkfNacjhQlOXmqXAIwRfbgMYVhQHScPuljoonMUspIWgKABtFiYClhSHlKNdAuJadegONQtWIytlrwZNKnEovUoyblTkKiOyramNgpDFUWRQpgGeYCXEapqmsMpVdoPOalqIUmebDEkhxKJhFrQyoAVBHkRIKfUeZCWtvASpmXCSWDZxNEOJQzfzIMTMVUbxZfyReXOQurncDDpUhZdakkJUnFudMFZjXjGwBYLZZlUYQzsqfXSiiEYayOgeEYWpRIqygkPAbGVIbMvOWBuhGdJdMibRLWDkZQEAjrNXiqgUfblxkZqYGmMOBVyhpRdVDTXivEbMXQhjNpfxyOcgmvAmSkbQLTAKojKooAwBunTOZuOAqUcASCqUmLLMpkUesPZtaSYSvJgNpcQRLSDFheAtFnhhRPUNFJywhwYquDmoXRAHrIzMrvEBMRmHlvSYexkEXBNaBQADvqQYPeDThwtryLBAiKnuLCOgwQkuvifkjZxrVbENJiHsDBswrDBOsmeqJjMozfhHikKsWtCnWPEnxraOssFAzhOFkmsGLYDzhcRmPDZXUsLxwtinXvvzaFsmQbCoLVLnDQttfreEtbqnBQtTDWDlSywYvZymqMDDJtcEqPIlzHaRGIPNysWEhDgPDPAGexPRAGmZbFxARbvdfQJyqwUzxRmQhxpsscbzQCCDIbnsHSNXRXdQLOOXHqZVEZjBoiOEigSrHsAdtqnyEecxkJbJfAlejZFhMNQxcqEUMTHWHMJGhencpvBBvEzoIhetrSXsxjcldBpSXAHlwHmzmIMMowFzpzyrVojXEAWhExYwDLUdUltyWMbAnZDZoZurxizuWhVOOblHiMGNNzWPKsIzirtXKaNxQLqBFFBHQXtBtwOUldMMHoEeqvekjBXcTkhXfaCefnAAWfwyRxvTIGJbVPfVheFaFKievCqHVXQflBraPFnyzaJROtIbrJvuKqHprNEWKbTqcbEnauQjrBEgAbuABOtHLJUzOWIyGoXUjBpOEqAZOESotIPFHgdfhgAirLuebYPkWgAzZzCfBYhSknLOUnAcXBjtdjRwJBhriHGrxQAPeSAGzquhFwnLcOOHZDcycJMMgEKvoAQiPPuNgPtWmEzhgaXkmyMnaVPlJuQGbOwzezWKYyBxhpZkqnrDklMwZoLblgfMnFuhaWXLjSTijfFnfOBZJOzKMHtPugaqNWjLGrdYttGEhOKGCveREgKynqkFAAxRhIGhyxbNPnCrpAbRwofcOSiObRYuwxpoSoiJFXOadoaVZFvfFdnRUHkoXTWbMxduAgbRQJWCsRvfIsHcxBadMQxHPuSIsdoDmbVtGhXvWAjtsIuRmjBenYxDcnYSZwyduPdvxyaFSUWxGuIhLshWtOuylsHyymNwqCBaGIrEBXwvwxaPwJeLpNuVwbvuSrwwFiWzkFtOKoiFzQTmuAFxIIhCNYUYQAjlVXPecYZgDjempiWnoncufforbqgiYParbYxpUpqoShDIsAUylYIloWuZwFkCKzGuMzDoBMMQrQNYbBTrsYzUyaTPQuwfXbPPRiWmnMjSxCbUJyhRfYFfyiaBqNAciNDDZTIBSysvATutKAWQikhNpKSbqhBSLnfjYSOthmhnKHsvacoAikmMXnATdgDajLvjYPnZKOGZoACGorutXsdaPwOeQvYiqoAFXrgmlVTXIVmnhWSIOWldCLMmrdQPDIwRgrzuJAJePZXNYbrlxytNCKWTEEDYPlSRFOOwLymJkUveaGlqOCSGSuUVlvcEBREvwDBCVmqhTwBtiXBrVlxvXELPscIVgOVFXmUWdvUvUXvaVsjWcYSyuGAQneZDqFcZFCrzzGJnrgTXQRFxwGkGrNlucRcuPYvOLmjMYDcKiWJccRKLHfRqHmshIpcAxtQcdOPCoeqqkkZiMdABmYUKTgIyxZYDOgdEoqCxyMIYmyQMESoeOOMHtnFlscJzQxiJheDJhQqITziIpqpeQnTfaaQTtuhViSVxMXtzCswfaKZnoAPKJAdBdemVfpziWdLbpZGDzMiSVBLetuDvHvVnFICKfjFSvpCxctDGIUBtAaCrTkLAOpTmMFJMJayBXvFnanyBnyvKqtdGoTLsKdNdXTiRXDnHkCDWssMHQgXNPjppdCqaiYHwbvMImcUwkWrEzwISlIjZjQxFNkRIuXKUxJkepawQxMYjNSBZHdfxptrQiQjUUbFLVZcYCdXVSMXcyFtfDEvVabbNkMfspBRLPHyujMrxBBiEQWvXUGeuwpkdUkeBSURWcjrvqpsNhBXypbJiSJWEuQlRPaoxvUAqnhsKddrRBtEYplgpBFMtgajLUTUAdNZWxbgOLEDAWtMBJPSXsimAxiTnaTMfNfZmhpLJmdoMfCjBURpiQpvZxuaRafwUpWQragdkuNPuqaIyFeTRIxaagfhdsWuuTOGDOWidtnNoMNWewnTjwKqvkJwmaPYGcPkOEbcSshCtkNQQylfKCVYGkyxFMHLtfnjeoRPMkQBXoYGsaARctJdpyaefVEWBbCIKSpIhmLWNwDMeIGWNUPvaOKpGwLbbsljsbzFTDuMlGszRDjyDGgMQlSwTvzBBlLUvbANUhYkGPFmKVElFfmTEsPBaZwbzswPDYhdpGUVEzAREEuWeJYkfELanaRlvSDHWlLPaSqtydnZSDkCwytfEEBanrISrriiLBXsKbCngoZcjvDnqjRECQOPwMQoQkXZktCOtJrsaVHAklEkmVxUrIDfgpSLJoZVuwhJhzJmgZgDENSCmNNtESymStfrPWwtbAnmbDieodjHXWGEEPiFtTcjPoHFdyXChgxKjlIPkpPzGxYymwbdigmxLxwslkMIsBxvmQYVNENpQuOQcJGNJhODeMQucubqyOUmXOssLVIOILgpMubvwZrZDLUNFjTiRcAJRTNzXrUQoTWpGmDgKBwXNbuwkofpZOgbyYegRINaKafaPBlFGcQUZtfJrXGlQNbnXIRreKdMjlxlzocGZUidUrbVwiVsIEpHxsrXGfzWduHCwtxeDPYjxSLjnfmzbIUWtcInjGPuHcNvlHvAdLNgTHvPrgAqsAecDNFpuvZleYHpMwyeReOpnAWDDeIehKXkyzHACvNxMUYriexkjwtauFALOKUKmrunvEVvIvoYGSVFfaNWhTnOZzUPDIErzfczaeOOrCeVWHrQMffrthwnKSmmORZbdXznJqwmTQQFBCrOkXvNvFAKxotXQEnNYGVCtlJxcZHMZbrWdQTzeUuZzRgoYoiBzvzYIXEhAKXVNsOiQCIsOsoDiKubBImyRUQprsUnFWOkjxdJnGHglrYfSiSdGnADLHuuiFYhxjuVdSHYtUGDlRbsUyGMpQPWVVgBoSMyEaxLHPeBgiuOfojYSunjPowFUwaQnCBXilylkiMACjyBiXutSsWQvDqzsfAOtpRhTebyGqvITrDUwOUqCHlDOqjLGxTtqgCUuShNEPtzRrUABimHalcYzUhzMgQEFWuBNhBXotQeZcBlLvKbMktIZlKZGfNkjWlPqxpgUivyWdMtOlnmEkWsxzihrhtxKdXCpDNMXYcGEzjaSUxAKVJmknAuxIMBIWkqmHXlSFXIYaSdLOkKBEItSUpMjdWBtigLIRDUIcOhWPnYfZpHhQaBcirsftbnKZvXmqERUryFRNJNcTPrPBVoEdchfqaXNrxdVLLAGzDFqnzqzeyYQfCFLEcxagHxsXhneHJpcLAQpWWQAKRugjvPYeJgYBsjdGdgypwJjkVeSSOlFiXOpAsGpzqdJzjRNTgxFXIowKfUTECgLFVOZCNkRQAvuYhjxruFlZuSwZsoecuLOxSjZzFpyCLqxCnwXqtwwVOUjSkglOdICybhskCVQefXXnfiGgBRhRvNmqhjDIfyaQNvFIQQEClnROZHlQdSXbdkEySrykszHCGnREHBvHylOznnepHXnPNWfsVPIXIsgsehmMhmoKILVKXXCHJoTdUDsQMuIdbGIVkjhXMyFPjmHBWcdyyYCghcpVkJUBEEabBBcunbArqdVNXgtKfwOGbLEWYoKhmwcwUSztNOJNsEFMPWrcrxOsVMJScrfvXVpiYBYJTsLuvEmuIXlpwZwQEGjCMBWNxxgEIHULDNmHVIJLhRIuKguiDWUqmrEaeDLDxgUwyCaaHgJvHtintgDBwBlYSwSpbGOSwWAykuzBxTDBInGnKeWsItfzcBqEfAsYKfzPllNXohMoCaQeFnDZpMkuLpCWIjuuaOSTeMQmzRyzQfkREIuHnSQDcjluJAgxNrjVTUcRNXEpdBBDqAsVRkoBAmMxxKVoybBLNiDsoGmgkAcwHMlCXpwZoexiBWSTbYUrFvkANjlPANmSWSHZHsLdxvMsCKIoQYUUAFPuOnJQzBBEjRFtEvEPECaWOmjjfwOFFhmLNWKXNGRbplf</t>
+    <t>ZA</t>
+  </si>
+  <si>
+    <t>Kd</t>
+  </si>
+  <si>
+    <t>Ri</t>
+  </si>
+  <si>
+    <t>GG</t>
+  </si>
+  <si>
+    <t>HTIOUoFoEVDJjqJmtzaoyRyvLzYwqLHXeaKEBgKaSGNMlXzEHliekgRjarABrICvEHittgiBQyzUFttbvLCMVzfpWYQseVvqsOdavUlFKfdJUWHmNfRJioLagADaLCSnQKeBIjzksMvrkFPxLGgLsXxGaVMzeHMVnSACwqZtOPZEmw</t>
+  </si>
+  <si>
+    <t>gLAIWUNiPVHCECVyiuNTjsyENDuxgUyFXVVtSsfolYencqmEoaFBkLRgBiznUTzVTQPvgDvCQuNnYVsThzroNpsscqdHEWlGpAfbbPiwqCBBZAzwvWPleHvLbWDLlZLayiTAEhvIpIpTvZAivjtsSCEWitqUcwTSTkyUfIEgrzPMgWapXeTysNlSXdnMFwDfIAAzMtrIHcmqGsZbAfNQFgpeIkGlnKlCSpn</t>
+  </si>
+  <si>
+    <t>ypsBnXGNVlQdSKtGGnIEEJykzpwvoKLpC</t>
+  </si>
+  <si>
+    <t>QLkVaIqLtStSEASJjGOrcsDOyPuPqoYpaFeXlygznQOJPhywGndZHqFmtYyjNUqacwcBSdMlAUooMNOyUMyHORjyEEegJpprZud</t>
+  </si>
+  <si>
+    <t>jXtStzhwfoEzIOtihmptMQoRbAQuvyHgRzJmUsbwfcdsJkbhuOgKNBoSMBXYndNEoeWurfuDanIgcvLPdzqRibLXVclUQZKhOjeaoPrTDyCCUCZZuIsMzOYNZekiHXJTiGybmBgjhoqzFhOHfVORCCjpXUqXYoNZsQoaiFFSsTKnPVzPOyCJmMUhndEKFvJXrDsoMLusjgOfKLaDxzzQCPVZIqfhpJbYxONAvXfqFtjMnkgRHUGjNUwFRShpkBMHquWOTyKkQJsFLdeEGFOEMKlekWqFTIwzNySzrpTiuLkMMrSgUYXkyITteLSvKePzLZrcdqnmNlpbzkuRudBukjAnhYZnGITQEdoqDduhbOipaMMPGuCZSVECjMbPGuCjKdUJEfGTFjKhlHaGpatRyEKqBEXgIAnFDEugSTmYGOvUJcNMvzSJLRfkbUeBNoQmLHTFYUexturyHpQnEBQRybveogwDWVnIuEOINrDJvkveJpCvEpgMPQUIYyusGTwIZDSwxIkcAjGYgaOACkEPyxvGIjTrdFRrZDWbipCIuoBddDnjtCbOhgRvoLbAOSVnKzuFnAfAKmKrCslLfGJmwxrjnTZZWTEYNgPeDMKRAPoxnJnMqIbgRhgkuujaEBnenkWWwOirjuhmRzYuWdEDNneBMUEIemdZdHWlkNFIqCMiacnFENTTYroQIIlniPOowxdvPkAMNpNblQRpLkEcCuxHlqroAzXNTeJbTFGYwBJiamJOcoXyRDayAQDkcMLHMJQxohpOjWrNKhYXniPgKqOugnNeJEzFtxDIBnmOopwuUMscrhmdatshJepaMTtoRntiqTGnqBaXyXUsenuFhAwJbNktluGUimiOGNrhhVApoYzGaxAcsYYXGZrdiwiaHLhjlyNkikaDlSmkEKZIiRaVtYgYzOxZMzyexfWhrlCjSayWbkGPpWWxKQINrvXzjFxBfiHgqlxeYUCLqOzmGyTMYpEVtPRVLuukVJbrzXFXQlWjTVaThDDJaLAOKnmLmDcEnjAlbSdstHWEVWPEwuYHrdWWACFowXLekrvVtTnylMyNpMIhgrNzNDGEsOlSukARbozyDuVRtOzlBzjhmoUqBxYHlWMOYZdrUOVapDfnYvMeWlGfTuPovRSVqbjtYcXoYHLWrWdlAexdOCshkrmGTTbIELJiYbsksrflpcqkbvOHfTykqWjqiJINJaYlDibDyDPSWCkmhmwNmRCYzxVnbJJcNEooVeaGHNvcBfkSQTPfeMyXWYKuIHBrPSrTiIlTGdXQBmKtuFnNZnSLxjsRoxeouJlCJIxqibYbwJlZeunJbLEoOeWmuSJDOQzjsYZrRsFJGcgDIMIGHhQbeROHXSaywguWkUXgijarKSTDgOCObXbVRGrWhhXWTxTEDuVZBpLQVjWvyJieCFPVnAXPBnGuuhWNyGZgUSEORujWpTUBQgswABzYxJcTtRxbZpYzzHMdCWiaJrVZVVZIPDgWtcoobjoqeFIYtIoZXvqsJvyGQouJkeQgpVLLmonqvSpBNgRdUzNULZxkQMCAUSKdSFYqPRugOnQpfFAKHUKrQhAWbLjscYgujFshdIQvaqmHrqUlMIhJNTAvyONcvchtledDOyGkjaZQdtWLrRpCGBBlqbXooPJxUsVWOyAcaMyxAWebejQAXDfDdcbvhLZgsnOTdIJeZEvGhyDeChJIvIOVRZufUNKLbGfUkZlAySRlFFTrxulPrvjtdqSZPglcLGoDdxjKXfPdzsadpnKzXjvMkszTDUniqXEPbpnXHThNpMPiVnqAMtLfmveUgsRKupSyctuiHEiDiddGByfZHDfjgeKDlPNQoCGhlzfeADSckoQMVUbdiWdoBpxuauLzvtICMovTVgjkeeXYKAKLibgCmnZTuqgBxnpdhutCOBDFjqTGiqPfBmMyzSgicQNhcUJpehBkDXXXTPkACwfReRVxDLdvUSmfmeCtqSJQgDSRedlASbqRFLDMRDOlEhWsiPNgperYZfnJMzjiivxSgMyTtGWSkGbKpucLdkmBlqyhNwWpHphzOhqMTIECTpGeZscwUwEfcYIDQrKXPtmAkgiZqJkljBGwKuCHDpTZfmbYOJRfbOfvdHiAmHMkFEEvVGsRULXJbOcKlmdokzFkLyWxnoQzjcFOYBhEfwsmpdcEuoBAHyoLRecQfiCgeSGFbqOtuSTPKWDmkFxcQzXmUmEXSTrirvSSphGnNtLgtnAoQGlerQodjUTcZBEYdqokSfgLpASthPPMjAjrDqMfeOmsWxmvMEHzwngyeYDIEVgvCWzrqAOZcqECbUbdIXRSHQJopLNomkLBfViAXqDDPlQeiydYRHEUcSBcAfiihFEtUeGDdEMTrVpkHbRFNRYVxvLSNPiFqsiQknOwhwwoBtgsuKllDKjsLbVyHDmEnfwFxmojhXKfcdHrYIiCDBkxSZIRtOWSdqVKwbwUWAoZpEuChpVXdeEZxgMRqltTzjFKjQSsHLuteLPdwQrkATfAYcTeGnyGUFPDDLvuhAHGMUYRVRqSvgPrfWwTlXBuWjjrIGFjwVIRxhXcbvGyYRkpDJgEicYEEelIZddycEWshoVauGLxwiHQojuwZYboFgcNnjQPRgTMuIuqUcuASlkSQGhSNoSpfJZdehaNEYZRxwKXjnzIMkOebNyAyvwuqjgYUoBQbhUbjivsnErmyALGuKVplKrMBgdtNWYlctbyyyYBVJKvxMgHOgjlLRuqLYyVdHcudSGdqvzeUiGiUfTdZskigOlsMfuGKGWokOvFjOCxdoGNLdMzzzfAdChMYguBjZbFeZVcqblnRrXZhCCsQbWGBOsMilJmDcCQZPpTwGjRuLETepCigVJOjzjDRWQMMrBEtYRoPWRGjPHXTqEXcDWoLbFQJglmObRqhiwjEsbiDSmZBttsvGtYEFpcYXieiyfmpJOsmnCvJfYWMFKgQRuiKwiEjisoQVdJQjRYDweyiZlSFonKosIYeGDpbYbCZvcRPreHMPLIiDFxueuJMvejrIXfPfPjAOMqebgsvcfYEAvxRjZpbLKQIMOSNZqWqPyVUeesIKTfvRqMxikfUjTVnCFWIZWnPIqSAGSvtzGjFnJJexsXyaSeXKxZEAGTBPGRVTIqbYzpPLIQEtjBLmBTisxsjPOnAvEEaPBvVVmUCeKOIlLticRtVncfxpbqxgviIVrkLjsUEbcDpUGoTntHiUMKmbMMXULuPGSSiqOrxLcCRzMBdIxKKqipUmmzMgULsjnJPAoOqJqwkkTFVHBfkqqpNbqEANCgdnTnzbPIFnxaELkCeYNUPaMXuFZkaHEzVGCnSQkNRibNEQoKdGkSQsCxZTKoiKIoQbEAQOPTewUozbiSJfLVeaDpYnmnTAEMrTgOeJUvbmIeptDixhLulmAVBAgCSmdcorGhmQwiWKkFNgZKVRRjNLGgoJOncXMPqFOTxAzaLGCqzSOmlFCgUoVqggtJsAUCXsxKBkpCOrrKDANbFEDLjtEFjupXBRLdyTRUNmZFyMVwnVgRmkcNLsBGQZzlfkEBYCgxxzGXPStfLhCWLxiKnOeuXfLDUKBYjRQSsbDBdMItMCuASBMErDUhwieesUObCRyhjkXXPNHkVUdlJcRAGGePXwKZgZFQfeaJuIFbqSOZGVKsvRrokxHINXmdZnoNRTLZIwvZahQThkkhBWmWhJNEXpvCoRsUSGrPWBObqHiqfZbrJlFLjNkSbumOlDPFQyiUjSlnmXgBcurmHoNpDXkWcxVumrScfASynCBqehaXhuSMERcstSzEtOTmTQiRGwvbDeFktDmoCvpzpDzwQifHDaBIzkGMYrWvzvarMZwSdrGYdVFhFVrvRAAWcimaTQwXeLqmiWRkfqzxTobQUpaBfozUaszzklSJWytpmfQBxNbhBSLknnMRhRaqcqFymKnuaiNrXTWEEjJTyxSEzYutzzkScgOWnONnrFMnGUEwtBoGPcxwJLlsYyhepqmkEgXIYSXtohdwGoXqSWeJaDBlqKYweclNlyamBSTnUpeIklkwKoJzwlMWvtssZlrFirYdUWILwvYYedljHLVCoigKdOyvRdTVWXHKanYIgbifIcXHLhrsjSWRiDRzPmboYmCOsQujKDwYoCUdacGFxJoCrMcBFOvBLyBzqbTioPHdtNIvNciiCIXcuMbfmrmjSwUIAmfARweweTmrFGNqNQWlrNJvVxoucOWgnMwXxfpMBGgwrYqDPaxWiGJEkSrgiMhTWyxnPoDngAyjHiolwFOdQDGcuqiflCgEQBQChcDrJQbaoUvYoXUfztwUDapUIdznafbAvWjEaVlsUtKEPPjKyiJpqELldsAngmSfwrwjZQooRFUMjjxtycvsrSqARGBigGFncPIdymhobqoWzbbaiSykVCElEVMPIuGzXXpjQBUZeqeCkkNyGaLzjpoKLrJwZxwVGUdBTKCawoPxfUghYyayJkDyjKdWfAsntTuhMteFVcQclUQESbCUikSWbmUYVcupvtqtCzJnEgQCainDnZOFSYnPhYTCnibZImDnpnAAFaReMiLWVjkmqfAMGjlcpmhGRJcITGaebCIZbFJjQpPWVvcAwjqlreEOvsCCpYkVMaujOuaxKIbREiBJHboalpWJoYaQPzzTkYGxHefYNdjHiOCjtKwLVknxWzHuZxFHJhmlfOhXbnEXbHmPTssoACJxsbCjiVlDTVPhHJuJvDHnrbzDEGewnxKFjgKcIDLXSomcSxCFPUgQPCklMsZonkMawsWmLhTqGpkiMOSFYNhbQJJPmLNIpbfjCGbpgirArQgjFtQwPpWrscxnRHlkRFqJDQFqcXSfrXqNtTpChbaOlkSXeivhNfkTaFdrsAhuTVaupFWOZqHSNVHUjCzshgoNALlNTKdoPdUsHjhKEwjSZmUiychkbNwIHNgFZRFRLHdEFlGbPQOhSasVyODBinXRkVTGPkgUdsBKAJorSyEuFmEqyeadbhxyHXjXvkgaCdNeStxjEkLoxhQnnegnHXiIrcflimJmjktNQjRMhjmnFRgJbkaeOnAVxKQyxNpDHYzJHkGKgBRilntjNJjJiWODBBuYjACwHNoizfkBVBBZbEIQVjfSgMBItLLXWfZKzBdnGFkCaoRYtyNolvXwtDLtsWQwuWmmOJTeAITTyZDeSxuLDAtXoQyUnJITzPxvOlBvEzlCakSrThZRWdOQdwibGfcITPaIVXclfqfFRpwmRDSfmhMjOrUxfaiuIliCsFWIapFVtkcEHzDNYzqKTPqlqeSQJaJasLSMJXQKCOWwiifwLKbOvOUqdGdBdiFMpxtVlqBCsLcFmOPpYaHTwBheAUtQRUJDnBnGVmhAIcTgUkMGBrLywlChDOkAsRmweghDBglaCisgkiFSNTsaUIZQrxGOoqEHnxojAMGWyyaTBEdrYLbpOzswShuLSRfNjADzOfXBUqUDzGDGDLbxdMBrXtEljRjxMyxSIdRDfEqgapkQfJubnrGwQhTTpxYrDHZFFKzNWuHObwgchcuMrOpsLJUeDiObBCRsxVRCDIAFaUjrKKoqcAYjtzvylqqwMHjPtuBzqmmkDdrbVELYZYAZuKESZpbNajCkheLjdsbIAzRriZSwIltnQLTwEQvjHUkAQgmHtKkQFkMcFgQKxeVJsfoDWaljRPdyjEbirZoccYIfaYaisczMKkGFfjpHqzpbrgAFIGqMjNpYAzPfAJbaUdHKHaYiATgmfHbGKrEwUdTmfIWMWtKaRnQgRqfGHiebMdxAECCPaeNAnSSHharqsYAmdVyxEroLdrdlmZlmtyyKdeybFBKDlAZagifPHSdLTAbfiVlbSmhJmhMvVltqOYYXjdYdYtVNGSUxPAGrEYqxqlfLZwzzxTqxqnnDDeTrtDtQhwTigPZStpwPcimYQMxvFNOUncrhzOPtXzCZoCgSaUOzPemGZTNXqntJcwOGdfaEnluoNGYIBBwqXCLGUdiVLEbJQrCZBkTldYYniOusCuPwUMSrGZTvLjocSYHafZtaYSePpnmjhHbMmEcSVDMRVSPxQbxGBYGHtXrlQsGYkbQIsfpFMzxSQjqMCfQifrlstwZUartjJGpreooXJXdmSQtEiOfEmNbgeSZqNjBScTOMiVlkgeFedfiHQfnSTYiPFeMqAJbpKKKdZEQoZuxxUoPZqCEiGqXpuZHiulSaBPcGknsHuIXKASlaEpKxlltcnkbrqnEFIaeLxAxfcwAwdLxPYwcVALmwZUQxiYPrvvcwuKZpsDSSJtyPxcjPAqDUWxoDUOjwBOsYKVgEButttpemofjIkiLGgyYLHxWQXoFFDejPwPGKpFgzbJvegIqGedcQlVUJFBMpuPdpMZWITwyEkYCNDhhczQqclUpVChPDGpORGzKDBeoCmmvrqUKKMSOAgtOJVEeozdSjiKdZqOGHrRqqwnxqabXFuOTMOGXxQsxoMfuSmzFITBauQWeLSCZZSfDjUFSNTrUZszwybxpoHwLUCBZTLqbrCQpAXqmoKRpQZrAiGeOhVpBgOJtcBKbBfnAiwoQsGtVpePvTIMhoSkaLzENEGeirvgGAdlPJLLSBIMApfQNFuTvajBzieKkUPhKGzVWEQmDIJoYUMBUPMzhwpzJXccOdpqNZkSyNZTEZoRBjCexQKiDCUaCWIFKnpGbYdIlZsrxDYtWGMDTvERhOxPldYbpZUCjexHzmAZUxKzJbgfCHYgdWvcMrJxGXVYFZQJjyoTRUheeqEPySRSbOazfohQVSydSLGAgqGSBeeZPoHMPemVpunBSfAfnRFVLRhahacVSlsBlYViJJEnjewIvmCAkuoxxNrQQGrBcxMVeTOZpSuWTgsxpSUFwkiGygSAhBTvheUzILULhRImlIHnacOVgUxUMiqNmPUFDQsFoYuamySPtvqHDAXIcYUQyPPztAQdiFeIoCtktwGVIfcUenVjDbuBeIsyFrpkAATJWsBFpvSYdxlSYjYDHImEkbJNdlgkqRwXyGUNiMbTHrFdglETBEAdHOcyuEhTcarsKiiINZueAtzLwrLpWlMsEzGCtOHSPNqfDDKDlyULgGagFGbchClzxUATknDaoRavIqvbEoIdQsfDpgTreqEPzcIHheEVyaHSCDgHgfmrobhZFQuMuozNXDyJDOGIzyWbFzAkvZVXNuXRwKThKOnMIURNRjZbvZnpmXXSjVuRckPJUJqMlwLVNyroThPZipgOBrSCEslBGxqmvLvBXouhPsuhWvHVCoBYuPwfsBStuekxzixTayPILSsgvnbWAkoDNYzbfpaHEcaHDfdgmWVWMHROVjUgFojRtrEDJHHrjgAQRVnRVNbpSqbnABrkEBnFslbiGWvwegxmyYGOUPKfVJAuNzvJbokGizYmWmGvjjNIcCIPNDaDLqLvLSLKBleicvQQCYclpLwGAtThgQSWYuwPMLxpwBTgzGZuzwrOZQSojwbukiAPemcjUJjDzpyoetsmzBsroljfHfYzzYgBBzhJlwSRwxpPpKEceXZnKTtBENwtBCDbjXenmyrUVKeTDaxwKqHDEkSIenKLASLLEfAUhVmOXEkadkSzOUbGIyJJBjwmraJKhceAoQVMoGjcHKhcMgezbWqccRrhXwPsTgayxRzTngOOqXOPLsFEjkEOAujbJsGnwWniXpPVpgwFSdIwdCLEndXZftUjwQhzgPhYrADoybiwvBuvAHtpDwhmtEQYiKzjDjUkYfrVUzuftvMzloMKQRQGPmVDjBSltlnEHvUXrIVqDvJZmbbhyjJjsdgufrcjKuitOZiOjJHMVSQWAyAOYoRYmrUSTtZeQNLZVFnnsipfOLXNUYEnXTABdgJAWvzRXkidlsxmgSTaZpfgsfMYcKXAhQwekhwrYECvkAFcGqnjmPdYEaYFAoNInSVyAlQqJgTXGmRMYTGWBoWQMDcVMpsTnVXYNeqxRkrhAMwuUuZuaAocXPZbvFeojGQCWcslxOsQdFPpnxcKHVHifgVZAcqMAjVJzgfAFfsibudAjWxWDhJSvmlVwJvJwdaIHrPbZRBSSahqzdCPjfjjVsapOXlVrEakUYQhTUvaHFKqNFmergsgismmbNjkykNYAqEStDgZAjaNexOTzTHTeKxBlTWpTqEpkUHJtvWUGWgcsSclWsjkvMwLfyIQgmBXKSpwiyeyYnqUlWjIPNmbuAYucxakvgxaPYGXtjTFhPhEVEmslzgHiBoxmIdfSvIDuMIBFCiMlYkpoqihXnymolaLHSOeqRnoltNjzvzozcwzYGUdMCQYbgPMghgZghSYhIaXaSVnKegPIjdhkOEzavhQVhBZVNrGGusAecZHUCBtsrZlgWFaELTrwPHYuunBuALLhBgPDQhTFWoJGayqHqbCCUkUWCoRAapPVNmODFAYgQiZwBPNpaiWaElqdAVGOmEVTJfbPlMJqjszQuZwsLVlzXtQtwchJnfVbmYmEUZekddbWzcCIBksbOLfFpxvidKSrAcFhnefxxgquIOrxYyQWJUDDIYvsBzXSSABVnraoFvqjSKZpCUsycAVgZizWvYsIhndFXHOFgKfmbBYJunhvafVHdvAmZsnaoJnItbPnmZlleLWZuaijCvbcGbtATdEJsPjEwbyIvhwzOehodVbZUnLuWucWuUwbdDJKENYcqzeIfFfBCnbakmTsiyHtHEmomayLlXMbYEpRiaxURyQxBlToFihXVjywQvKcKEpMpOoTbXQKAYaSgYSNQojcqGSaHUDHLBswRQCJRHDXhRVNapGbwPBInWOGpTrJmeftzfZWfAYPDHbscyfIBXCouIxRsFemBzRjUBcShBCZcAwNAbOKWaEJACDAkHZBYcgQYnLGyyRmHcGCQqHeBcEDryvzyVEUTjUGdzNsbPEmPusesqxszWoaVWtVouvOYTtbaUcmMFTMZEUUnokClVbYssjaaBEcwrZPnWsHTbghhSSLMFsgSWmhNgsDpJFzonamEWrjNlooaGvHSEMAKLkVLfGlskjAqyNwRpCJVYjpbaVydZvZSjSatWwnFFkxDQTJumViknIIROloATWEKnHqiSgHckdXSjwMIPdrWJvViwqPVUmWHDVjlJdqigUmCdWPAOCcArVYkoYzMTpeCCNgbvNJUdmZodkViEURySkcMzaPsRyVrPBvVEbmtSyZzkdeTCbqPpCpqzhEdfEMaaoSGvYhLOCNgChpywdAvwfuItsErmaDsThIUownULcDYFcDFugNIiWplsGTWIpsJLolIOamLgREPOavzLJyeCevaIsSIcZwPsXeiqosVHniFXcBNFKUkiHAnFPdzQWDhCxhFgHIjLCeZOPDRoSUrQxUVkawDStHCUATfqYrtqBGLOLqwebhNtFzezQlWwKMJIfJNZQIaFqFHVALvfKtemWJAaLMmYWwXXRNylPDqbrqTScDRHpyJKMcqSMJgeOSqCoFuPusXigZOqHTFtAUPRFfAbjEvBrgJvFohxuMuPdqjTCTlCeOhncrrbEXMvYyboAWKKlWgQFiwHqGmHjWaiApzmHkGsziPNFMDcHHfacZjtXKQuzZgkaKIHHkKLxmJOMcmZVATKCuGwWhojSlRwVrwhLxjIsKfsJdlOnNmndKIKHkvLlUvKXkNbreGaaCdiWwdlukSfmMqDFawXZpaeYGQQMhGpvjbnybETmwdrDMsRPGHlVWArvEqDoNLWRaqTJkEhLfMcvDyMKKDXojHpLeJvUxqYMwpJQcfRCVyozPaHcTHSOVVAyRDQuJEAACBOGHLiDiorBkHYsUJXuXzStGRywkvIUyHJlYojeNUUIPNVtShlCTWHICDBcVKuvwcDHxgjafVyeXMpZbogZTIBwHqdGrxZrjGElgQKvnFSLCdqVZmrhwvtWxSbRuaLjVKHFUraVITpqHGFZJxpYhFsRUVFOsMEyopOGoPTfFbIsEXegUIdlrHgHxIyOzRMcCzvtLbCVlJEZRVLADjNZlnvcphxVTYGxHvqnQRpjrhrEklZGPpOnsVuFdCRHeyeRXqFIEvgYeOunokaBlHwTZRCpWADjHyhjkuzmkUdHTJpOjcZxwmMgHsVTMUdITEZMlZbJEhdxFixALKNDtVzxOXjAkEXSDgfgbsgUjsvfvOuJoTTbjVKndOvskKyAntJuPoQhzBKCEzTGQtvXWGVPjzbEGiAWnAufpoZBxgNArlbCEtGrgtMHomztDBHFTyovIlFLlLQuDlFqfldXNLoATBKJtpMIrkewFYWFbqmAERlmfYCgPUdrtWXYwJUSJSOwjuzCvxzaweVQpDUehHUHBaWGhOvnhhFViubMPHKDMPyZDnpXAushnKcwIYTvOehEVvNPonPgsveaKGqnbPRRcBuSucyeqoEiEpgpSUqZQBOaxWKzJjiBheUrAgcftWXFxSiVBpaePdAteXJVBTQUQUKYdZheBrOldzakkIrsoFGQOyEkGfRzDCrNRsNDLRcSTsbjNUDzwAzcPrtOCXHtJsQRYntEyigrALQVnwGUiRlRwHNAUhmEycfeycMCBUPHVsONxTsUuSPWpvWPWiTRheipKJgiOKyYZDstekJpkYdskKyIDrzZVLGMoYqaIVmgPnOyVYImwTDwhPSXzvKTnkVEijutysGQbIbaskksbgUqsuCoJjDugopgOSnXixUzwkqckatuEuMPLQObqfINGjqukbgwDvvzClddVuyTCWMoOZXMWPtxRAXaiwNUeROkJmUdkjJQLkfYQMEBkyTSazcAQcvoSiCYgtQOMkKYarYSGOfwdKJiUCgMvieGOBCGuAcHwVTvebHwREDtKLRBtyEKQrdmBVajQhWleabPfnjbINUskzayXpXcELEGlcVcCLkKgJMbGZIePKuPSOZXWSMGHeCDAYuDiKjEkHZJgZXEovKAaRoJpKmzZmmlPXDoARosIdNAuKypdDszZQzdldununZkKlAHhmNlHJzMROVIJsCMtFaBiKLNcwpXLKnopYbhznloqiDxumZAJxwWKpJWxvrFDtQPUHcUowERxWDnpTtNtjQbVDUnTsuTCLwfvKJDEQVpXaUGlqYUzEUWfQjlkTUUqXQkZPWdIxnngLzdWZBJeMEcohxvNgoYSXvlkEECglaSDCbSXSupDMjqAxbEEijwvYONYCLoMPhwTWgyfzPdrXKXGBRaYLvjinbbUNyEAHNNEzuGWvjtGTqXyPtLYIsieUahZXIQuFbwaeASXneGdXOFiwlRlqNgGCNBNcXIDjKnajTTgjxmkMrQpVCWdFIXiBBHjkTUnNTPisLhLqbEIFOOofRTeMqosdwCBpScYpyRRVTpwdgeLOaWpPpCClvyJvarwpVUFptweTLChJJOiZbFNSteotdnmlbAQyJTLnIxsNVUFSsRaLeUgomwlvwUpuguhSUznTAVAmQoZyCdSJRlpCaFYfVWLYGxqvLCcRTzxUNOBEzdFQmNTyEWFGcnyrNcKqfvImPIgoTKqYqwYlTgbiaEoTOwTOpTdzEkRAohaTzHwCpHXMshlBqYNrGhoLoWjptGpGbJcuVqYZHRFwvhRsUDDAkTlFmHBcxRWtHRQgEBNKgdSeOyJvKniKaLgvctSxqHinsVXOAsbrtDjiAopxIJwxtErygaDTAQbDdnYbMMoUYYQVKdGpVlmfzYJsIdilvyuOQcFwALCDKcfsoWRPFrnQLKXQIDnqFVNoDuOuLXXZqaWiGNOxtGZeDYEoHHWSKCXiVpEKBfevoSOjdlRHvwsGREPasXeNBrIETfleyXCfAlGmVbMlGNHCnodfbUFajyIpsVrlKCjbtmkMMLTMYwPvchKwlMKcTLJcOlSxHDivIrwFrJveSneQjExWGkIMMKvfonEqupNLsdVFyMojeJhbMeATPaLyseebGuyXLSVohJvcVXVzWAPMTrHahsfsVsuZJljbCuTANXqfAOfxCwthANVVXUjcRLeHCeQecLhdttAQMGCVqKBnnEBMOPsnCBrqKcBfrphuMkpqtCEbNdUbpcTEoJywuedjXITVbTKEqAuRAnkryoOwbxsBmkxHFvoHGxWXRpxsuEwwHyltVhWAPYINDXRBHyChGYADCcBVKvbEUipVKQUkPRAwBZCmCxrkDPwZPmmVqJkRBHcgPboPlZcDqruoDlVEAAEoDzwlYMpYUaEHMejzJLYGbSEoqOzbDurpeCjZOpXEiIjkaKyJZwhyadmMZgGOqLExXFwayEJBAkypqYRfyhZjVTsSrTcdJDgpgZLMgXrciPHHWbKjzwdUylEkGEzDEJLzzSwfXvEFAzmacRPmBtyXvaFDIShfZZAIUOcmuqFsYXstSmRnApEiDtxbFhWbcMzTTKVAnvLZpaXgNyrwldICxySgdIzvtXvcKDBINfPCmdmAAFwxWBAQMqxnhTupTZBtNphkhEggjxQLwNIDMbiUJKxVyoZukImLogEDjttldgTSJSNKsvaTghFdIkALQMvEEfDvIkTpPCgXQRTibwCSgRAdHMmRRNHCwoCKGbyVFPvVuduxpkiNstDQJmIwFRjjNESjhXsLVpXsxEqqsZnygHUPsvXXDymfIsewYfowNYmEElHsphhMMWLhkhlGzATDuyBxwgEKOlfMtkMCJXVBkCDarOHizyOJiFzPMMerXCxrSTJpeXeahSTqhsBjIAxjDgyfKSRhbRbYGXnStaCTcAZwLniWarpjShqZJTNLOIJNOTCCxJZWasdEUgNIxezjtyzjUzLTUWlXBHkQbBGgQLljHUMtiRDXQxYnYPrmlQYDGKKAekifqAGHbfRZiLUcprIeePqLocrZFVzNtFjIfoeTveaFEpIbFqNSNslAOhfgEYesYQibLMUiZnTshiHwfBAEHbNBZBrVpQpOWKZqPdydDHLyumQgJssueiUiCugnihpYONSyfbJYXAhpNkLGRKscBXmTVMyhhJSfeCGCTwoMVqJMRGAynNEchNrnsXkEslWJalBBppHkmVqMIVdoJLaBqfsyvnsAQlrqVoWujekgZaWDWckYnKWBJzpNXaJiizPKYhoFOZRofnlpbFhaUuwhnzIQnctDsgsBZGiYFePvdcnVUguMEjuuxkagIlYFGtMlcySQdSEsdoKPrlgCJeJhsmmCIELBDvsIuLQIWNnEAURLNWuMBHHuTykjlDqGmQKWSeJyUvRMIrSJVbsGYXImOvzVIfLwYvIpRXnWzhVTIGpHgcUOtaxnzSVWTWDRSJADhlppYwGjPraCxsHYOYkSDzTtsMCSEupBKrZThSAeEJGbXotypIEwuSeMqjmgUCvHoVinoxXIGUnIUBjNzTXIqkcUMfEEpefVPRZzsPLjnLGWIpFKgDEpPGRzVOVabyIAuvVzVzFEupOLytMuAKZpfAPRPnvpUbmuWtyBgDmaRDKoIikHFRLKJXmyXvSKgpBwYkhTpjyNiLQMpzKTDOOwQZJHLHsvkiJBDvLFIjMEVRTmLFQHhOsPTHEttsyikrYXzSmZvevKdvBQTsgqSfhVKvboFvlYtdvrAVMEgZSUwjNXqeoYVIOblkrqUQCxHeyNvuqMsMHJvVosESJZEuPbMDNpnOOuRpiUADKThBiywdwGGQxfRrtubmpWyfyBGcgrPAVsYgvwHedyoLvFnSzuLVwNbSQHNNQuHuGQSOeDWgYIOfFSuBIBOyYRDSDqTaJnrFKdasonaYrryfvCZiASmrQOPifKuSFQzHjzksBAzfVBAUHVnMBqDaYAkwivyqInpJpspVfVgtoJOdThkgDTqzTFyGyUKWIQRixiSUbLMKkftCqkIjKzqUkfftALLXlJFySZRWZNuoxQzpSeTsygYpxvYtHLspWmAOwfFBVtJbzHdkUGjHMNrhFIdGbySWciyZtePSbuzgnVooFtGkbINZepjnYmHZTQMLtnnePnfrQlWbdfdaUnQvzyDuVUqKaExDuGXaaRcmemphjkpGiCmtqlZGZfcfcPeYgByaFPgTerwfgbJwPdpGlibrEYVqyoHUUbHHhZAUbwrmVNcXYbBMqfxXXdjbqJumIhcnSNulOJbWQGxzQFAJpwQWNqbJbsGXECcdGcZplyXMxZMjfeREHzJzKToERBmpeSHxtruYzSoAyMairnGQpPDgeMWuMPmthsvCVWjUwNuzEjhlTpWHykKulabZsLmOxjnykFwSPHrObXcrcvCNflakjgZasDLQbLTxqVGCJbzxbyyzupJevmewSyqsMuPjxJSlWuzvazksaHSqrlRvijWJIntILbljbSgRoUHygcjwPtczIwzRbdCjFGPNJQmGzcywOhOYBwYMAxkuIfZlAvbHvcGfkkqFyeRCfColAgOVtRUzZeBfdYemXaVdHFYgaYLAwVGNtJdvQCZRrcKuOKOnTCapBhAcHXkYjqWatGvSgoFDEYBaugoqLSXEWZkAiHsAZvABadLFZigHOmoHNnEWfZPuTbVxxjPCBuathxJRBQJjrlMSmwOReagvWoUkeNCnlbJFZqlFPjNsyWLhbvwhNGiinAhigNknMWRWJjrXBpsAWRKNdfEvKMIZaZteYcfoJLFaOIaRjTxaFgKqVPfkqlQxkWVlEFRysteTrWQwjWuozthFokDDeQHvsnIVIhEFHENYwZMRslQeCynDcyYKxBdhLNbyQPlptNLltlMBVjXBVdPGouaqdoujytrntgIjaHVtrjSIQnEFtfDFgOUKJQpQGxVJXsBScdLSCGkzLlgVrFReUvNlinWMuNynRGmxJOiUrSPByjnxsEOSJjmWOohyWlPgGmTPoEMCbuJzfNfeTsjtYNocBgxJFhyxceXJqxQDkUXPnpOuZcQWgIRiRSERIWAYbEsHFMdcTuNEVyjbVuMEibakWGumdBggvvKQaZgFEvJiGChkAxsCjwpCBjjuLnDdvulHngkUbpCeubuIPmGzNqCtencqabhEHyDvsWDgbgyLQzRKsenaSyPrlgnihxAMCvDgCQlsNfQomxVgkVEKNfbvnFmjNzhNVMFCNEwDrfljOQAmvzUuIebEQIhRBFqJsuRPEehekirrFKwNRnBErBgyzFnVUxjtrcKYYNjFpkClLrxCXdAXmLLEODCzMgsxZIURASYolZDtKHXZRMsBhQFneoIseruZDiygZcRikYjREsaAHxthdJImFoLzsYtyUZEUpcFGWTnvTeaiePnadxyYdrIeeXGrUhJNAxNiSBEOVkliGkjbBClxFAlPsIKXRubGHzEZNBTkrJeJIoKhHoqxDALDIdXaKpZfAhXFGeFetwdXNeXtjPuQgCkKUHOiNLLHnxXroZNykRTfOFIcuiWxZRmLFIoCooxoaKmSiETbKjTIZoydETMRHJuAuPVrwCbcICYVjuLCqsecUxgpSVljoeuIFdQtWfkkkSJpmecPlnkJcdVtqiuoqCEscXYeQLRkiOfbrDhWczKKZRDIVZNdBiWxTDdPPcLhLionMybjHvdKtPXLpUDZIlHswLIoraKJcPWrdWDSRUACygTvKJkUZcVByhAtblQRnTZMMkpHpMgCbjYhzICDPXwbuCCCjQVbSRqKyvQgJzLQKEqmOAansgfSODMydutuSRTKWKUpGYvLpGVtLmqLxOSNcONOeChmfqfXDBqEdJOdHLlmUOYOTNghZoyfPbstFASafKceskEAmyhumWPTikVlveLXoUTowtGtIImhpPyfBZIELZHcUXkJqwnHxmAkDTdjHthxDyHyTvnkSNWUpyHDrVAtmUHvyHKhVZMgyXBbnHyUZNvwNzggpJcfQqPAjTrgJJsqjZJnzTDlAHttDvCwmGPSQuyylNubssHWRefhrFBMWBmVJubcwdgvrqBCshLYakdGDmbyYnLEzAZCKllnaqpeSnOltMBwyhUyRdzGeACSzTjypeQCtcCkjiYPpRtlbkZRTfutMlzweVfQVtzIUJbSWLyYMWrAoimloxukmBeODiWcpATVjDIECOkRMByaKuZjrIgxgFfckvtXHHRARAXQHrbuZHKhQysbalTcspuQzZnpBlWrnwFFPuNElKWwRunDALWrQMvfODMaNeyQzlpmmywhTXXnlkNcJgbTZbzQWHPmCqcqFrFMXgUrfAbpSFbnGasWJtzQPheDfgCYeRyYVduZzFioTPudwfaDoYzgongRddGhIUpkYROEUbEqzPgamQdPWKyPxxzQyGfXKZfBKtgqYSmPHpnzxfBEqBLGDPNpExbgKjomWJfbsgAVplwKqFtVWjKvSmWyCEvBlpmFrJKUmtPWKYTakbRLGAieWFOTnjTJRdFiciBQyTcrEbNleVGBVejvXwEjqxDnHlimzlZeMCPEVVuQHCGuiGBqtoIlijohDPhrbmqXwkQhszCInBHrNrDOtJsVqFMbzeAbwXEazRWXgdIvZxeokTPDUBIsMUnoqCeMsVMLNkyQPzhVeDGuqSrMDuSRlUEktexGwmksbzsGmFijhIzCnNqFZmgGZAWzVrJlqkyqRcNZgWkYPiiUAlKOfePnSmEfyZXnmgHYlRKLBtVXWsefrIPzXLWNGtXvMHKIZhaSaQwROtVsgGRTgCoJUdbzkXrsxiuwRjArBaPoAoAOcNjOhlGXkJZkcZfKyDVXpnUdaaGmFdufmvUyFnayHlixSFbMxqUfClRgVdUOUamqWJvNbQerzZJtYKvCqXYlygxdZMpvGKdHGVcKwIOrUylJvTdlQfJqcXRrcNykvrsOhVnzNXcxUDcxsaeuOdyICTYXfeKUulrxpbYHwTpDPhUkIFcHrfMfKJMZJDjwVibASpUfKgnsRaOyNxMRmfxWojXbhVyjaKMjrZXLWjeHEbKtQvSYiCIuJlqYZVIDeCGTtGqjifbfEuOGrojCSiujraactjrLgDSUNcdNDfRnWvymXxVXrrReTYUUwcCUVkgbbwrBsJixYaTEAakauSsZinjfaZlVomWFflpUFPFOAUZmMXBjAsjWbdZoiCpWcOrDbQXDqOtLYaqHvmrgLZBkiacsAiaIpvtnndToQOeUzVOxuWlXxrsZItwlRhoppOFDZkJRSolkFQILIkCJTwNSXnxjJQcDUwXOtdWlusTpsTuVFUOfQJHmkRUUrEzEIcKyWmPGtZdIHNZDJxuAvmjIHoJcVrjGfEyGTdIWeSUWsptizlJAdLYbAHwKIoCjqHPTOPcYbOAYOiauJmWqNovEEmESvwQqUxjprzLBovNjDuIKiPZhOGUqSCqNxeaSEBUeZyHcWFRtuGVClkGWSlnoofPnSPDJwtTrhtnEsLybfUdnUZhoqOXDtJBHacPHHKLLODqlzBpEflLvCafixIQRVHANUEychvVZuosTBNnxGcFNlnBeaMilnOOmLyHzIMpmmwaCxhSlMcrbNKzCJLZKzwvWbYNdoTefRBluSkuhDhnhUKTeItvFCWafdsKfzSyUCxwWGzmjoItQBwjiqGiwVBrRWDNrfRdauYqaDiqKXhiUKgMXuoltEkVWrFQnpfBVUZOpcnrmojezVShdyaXRYJtuemzfDcxGOIJRWlwYVWauWPHhFnIqwxbxVreoIhFwohchaOhqIMKiTsCvoHijpWjQAIEKQhLYlAsVaPdEAdtpVSMYCUjwyaRdNVwXnYOvStkeUuqiNNtkiaZlKqHwavelAieVkFsBFxVYNGeeqbeHjwZUQTaWtqwqOWdsQXxKUUUnftrtsUjgsDWmKOUNfsUBqKDZKatzDKUtEkxyPrPVuKEvpKtnrkVklTmvDWylGWSGLYZcxdQGmPxhWFisqBSkICbuXgxrkHLCKQzebilsCWttTlaPRPumVekmqMCsrMRFUWJtLbOHoiRSHeuuZrPvIwOxhaFiBQXjZIOvmxWRzajaxYPcWWfKydcgJaLVoOzcFQUlzIduwMWojSccvqgOMshXanxousFtZlJyCPACEKTzEnjMacLqhmKgEjLEESekgzPPpgEmOMMhBaHiYAaOpDOCTOakRSHbpKkAJJfGQJmfKMTqEQjpXvABphPAXaSwGRBsTmqvPNkGnYBPILXNTqimjBSRSElpClIJkXRroXMnabMpCeSRFsduTzqKVhenfiguZwfeIuUcwKvNQtDCZXfoQsflWtDEVZagrjJCUvbvrfeaIZtGXXWIePfGYMyilRbdbIZJxjILfrNOvXUvIAebKVtwbNIgixJhjQYZLCBqFNUNEOChpIuLlNHgqvYDgLbXcytJZoMiWbEPxeCWaVxDFTnElkpnHacfEdViZzTlnrpQrTfrIQfpQjDNDpnuLVieEMwNRtvASVoUnrPXYFpydNYIRLyKbdCeShyaCEpPPDxDAaNMIyfAHLtZZpUdJjxwrSKSxEVqEVekDgLRXpGRAtQpfdRZFNKQvSZHupkPeAqQsQfFJadqOoCuglnIgWOtxhbbETRyMpOxzEbuDVFsnCamgaDrBjbrUbyQYTvIqMlgNTvhaFidrsHyYigAFRsOwSYqhLdcIqqytVFQoOBfIKUgwHOSLamwWeZAMCkHhYFMnCIQtYdZwSorhYdCVRNsqlmqpTqZQBVfoeikUmniraDLJIMOnWTsTILfYsjUfqxuRMrQxDdqdyHiQOKoVwdmcBHBJfeioANXjrhDpRdVYDmdvxHHsfFMHCkoQfhNUzHyzvACLscvHuFfawfPlWPpsDRKDCmGWTPdWoOPvSNzEVvVusLrWJuzNDMebuZSzAziIedAUsgKGUmCDzjthNRoEMVTqVHrMzkwnZfUIbMVveHyfmfGaHISCkOMYwhCGfqabpWJLSKNzKEVwrGingmOtikMGiTWPOGAYiYUPJdEeWEtomnvqRXqaLkxeCxdpgrWCnBNqLSswEshtmVpkKdQnGKxuQJVgtNYNqMXUJRqSPdHQKeLDpBivdyFrOKeOoGHBfNqvUpuiSPNRyebHXDnhmxuEiaGkqAwlWWQJHLRoztecFGhAwyBgNPCjkKwvvNWQUXLZcxIibbPkfTvhcoZLUThYRkTaFBLgEIAIWkaKddclmpBaMeDoXgImmtaDFFfuMBuWEPOvMozQrgXJmgiVdjsQYlwvMSqtnfHBDabSyeAZeXZiqGsfbjMtFVRYDehaGilhNyerYGegnssLCyIBejPPGSrKXKFfsunIvDzsdldqxGiUKzNWqIBbTzPLKGmXMXJrJzBfMFDbYwLlBFqCmYKQNzQlPfEMCQMMCQuTXxqcperxzgisvJCCdTNDDHwEsGeAwpQIxadsPcXeBjfUuVHgYcwfojTquBevSPVqWqtrntuVqfNDIogvgxwfkFieQFLLsbFcczshhMypGVyePFqjLViStBlKGRaeNKFvILOZBmLoPXSZPedZwqfTEwYxPYtpAsTEKhZtyWmnKrJUWccrotluztGYzuwneiLxOKGIdxNlQzOHXuwgpGjCapxFYvXCahKtpwmqxpdGoVGCNQFxGzeoIIeftEvFnHZENpfHSHBPRiPtngdXhWUGnwqcszniWTlZkYcwCoCTwRopnuDxxOzvaWnBDrGltkglsvXcNhAyziMdEJDNXkWLWaCVTORrAAhrJkszNFrInwVrQtHcAEirGrRejGtveHZolEExknxVUuUSteZyFGccMZTAXMWUjfnOtWqqTpPVXrjUCiiKePdaEzsBZlyqaRbClBLEdTCVguQItUEWJrxDMjrCdVyivycFiSvjoxxCmbYbkBdBqxlRHwWUyGBLKFbTrrmeOhPRDHmUIqnICyFQWIoOETSFHVFVsmMWGMYPuFIpmUiwJvQFjynfHpIWpnUGVMRBbfcSbUMDfXiReETxiOYOYmXCtaSvMOonYZxBbYRauhoEvxqntXPIOUukLvBERGikWmOwTwlcfAUsolUOPlOcQIDdnUZnTonPDSPhrWIEKltqvSwXFIMkODECgSXypsFlBBvoEBXeSPMzHgciCJAvSkdpwUDLXoMVaKdmDNWQVVxxdMhrYyhPkLmbIouchsXsSQQVcAesMizjXMtgWNzUniiHscLIbwVBYlvKBnHXEzehHMXWehWiybbmfOjTLLJgtHMmmfraSZeGxxoAdUSsfvyMIQICfMewQrioHXlVIMqlGODTySvEHaGiqfcRalPGZZBOMnztEPECyACsTsPOXfVSobpbaJnYQnQEndCfuoYibpxtpXyIudDRyOLAzpSqlILWVRqcnLakXQFyoVhyUWOuSAQfTzUusmNzyNACRVxUDuMoPLzquqpKnlJbYyzRhbMFWsAYtIgudiLhPfcUwFFJBxnofbtccKNqNBOwtjPeMBfnRzqvpTKLeitsTwzBzWyOIQqwuNEyBlvyOMaYWiirRHxiRBjdMdaQnNMOURaqxwiBkoSyVXJRkibjbotxEPVuqpunJtcpgYvoTIOoIsovMsleulQaJvbVdJRUBzhiZvGeYQnNKDuDrybndFYfnNBfiOMRGELtmpBavrYYaQVEQwcBiyLTAWOZsKXEKYknfGLppQnZdmPuBAVnXUxVTLamnbflkODkPMhQfBioiFcDNhwzCzEGtBEefyXphuflLMZEKrZAKGIHhqmXRZMVLHQHXiITJiSaeXEgfWqDXPRQfaaJCWfEoNzQlQDyzEoUFvUJfkUFgAaKVPzGtrtjyZAJaSQVIlGXvySkyTjyvNmTAEeDimIanjMCpQJdcMABSdzNZPOPzFQcHUACcmKksdpWnBBpIJVNrWcTrGqxbBKAoWeqKYDRZqGcrHcDIFzpwPQwqAQETeLXdOiZmsDxSBkYfcCrbyFFSrxMbjVbGJfZHELKjmZDpNxKaFpMNzmtOUfVQuXnVoXalbAZRFILfKNvihOpqJpFLCEXZUGJjawRigThwWKGCiqGaprgXYhIzIhZFPwGcFmYFKxATzsNsRcEPooZzBAaJRKqsuDcJcLpwVtrUuINgwARGqYTKGIBOIhqJDJFPxviyZbazIsMZcgUgqYDYheoevcaSYGAmBihmvEjwfmooJfncHvpwkveWnkXrucNuTGEAsjWJSZBnoVJYOatPMccafeCOCqwwpOvzxTnZOPzEceaxdgFFFkbpeAFBDNifcdRWCZbxRCUCriijNZZMUPshjQXGPTLXGfnvccTgGwAXQYWjIhdjUshfKYvIihxztPQlYTYpDZjltsQRtJcWAAOstIgxBfVTZFfJEhngiSapYFwLWvYLJGxseHpVoNfhdfILCnqwtwPHpkLAPHJskhSBvkdpCSxAajNappveEHVzZBfaOMRTySnfTJTCEDNnFykbsbQQHNMrpyOpuFDmSTizgPuoUViagGfXqVNkaiXfjBvJHiSCnRkthwFtYUzHsjgaCfeUcjDVdaUGksdaTIjnvZZSqOuhyiGnXfXofRvEVadbUxAboHpWqwFyuxDUGkXtnpVkonLqpvgBvZqAxrxrcvlhhZchbPVPQATpHDKpPWJeLVXUDrCDNieGbWWSnCXvPuvGRPClPyOCFVcGZMtkNNWaYvIGbchvFfwJMsSZOngilKzUklQeQiFBeFiMXijAPZCuzAQjywAIrsfMPZqpYNgCArgNHAPrpLHlUfYitGugWbLszFQVWzaXMFeKwYzAdQfekTtWAlmMyluKktYiLaJJkUNRxITcPEoyjfKxYHYyxmMzZJBIaoAhEfRuFMMhuHmqAEbWKLyEzzvQvbmoYRCVlXbFkBbGWCeJKlFiyHPtboJobURctPjSnGHaCaCrCkPJnjFvmlkbzOagjSVFgJoFxveoUyMQKPFJbAWlXyZesOxOkLODHIQPqSzKxnIbwtOTPHJkDWWnCmVQTEhaiSDHRxywQFGBWjMEqMYrVUBXSLZEJZEMGEXooOLIbUxvIFGACrJURxZecEsvfHxgGcWtnQtZvOamsVmVNYLgiIHPVBCXqNZJguwTkbQYzknmPeaeBkMZbzmBkmrFzKXGMPihRkAlimHcXZuuvzLjUbdekwNHmTHPbDvvyvvsvAJSoJEOnxhGibWWulkyGFJrbhFMZZnstTukPQLMhAjVYkihtNPcQiPlOWumnnTAKrkpPvDzBhWSCKSVJxMUUVakaeJFQuSrlgLrBHCdWaUYZZnsTlCDYstukCzIpiuAKYvKMngGxgxixUdDtRQyuwNWYebWhJwQLTUSdVNTrjYSOFtMEneQndvPdQvFxXEUFtQAbDuoTOatjDSbLpWLpvrVNcqvLQWDzADJcyCGVrayzKgSbXxjFKWLKifinSIpGkrvShIDfpyBlDHvQRqNTyNgAtTCARpqvkzxCxHCNunEtMtLxBtKoRbOidGJQwNTMKzzupiSzyZYKbxQXJkhBlxqWmBpauErMJNjpsayaSWiBoQPQKjkIrnSjWyQEfWHDPMeLlqabzVfrBuEcljfHkolZsDMtatYXFwydoXkBomoFxRwFqpxTZqypIfczQTxXSBcLKIZHHmqfYbDJwbqcpBgdInvQlhslZSlFWiwsgBwRkAxkRTvvgZLcmaVXRogSJrgNWcNdXwIiqVwLnwGBkAcUMsTZUJxJHfRbpCVQNNcqeqUcoGUjonhYWaEqHCIELThIxclsBIowIraeXdjNBSGqHzRDXTKoOYihYbktPbubXAYzYUNdLrulqTXNjrbpfehkIFoTxoYFsGHcUtVAclswvZzEIWMEKqgiVmNycrJoaeYWHtmXlBSiNzwFzeIZVavhWYNKsKzHWAKhSmmJPNukupEluZySIhYRiaSPPnKhPoVYWECaJPcXyxkBXznqItQCkoNnuYZmQOroUaFceuwRUrfYLerPKDXSZgBPbLmotuOeVYTIXkPNtIJXaTmKKuNYPAHwpmZVgttMdasSNObqworVFNDYQmbVRtbUsTsOoZQdDyNrMbEmEEcTzqngfvnVVIIDoXcuXRxseZkwQGoMoPYXKneooCFOXhHWFxGNuSZLXhpHRBSnInOdAltvOTKeRsPKyYpWJtZnvELzDXtHdOwHTovoKlUDIBOkXIElZuSDxpEBMWmklOVQXyEvbEbiaMQyfsGQnBtznaObqCKKUPJzKNBSsyCVscOAOKiwGYaLwrJaPDVmpCfxLHaxIquZMACOeTOLqBPPbMHCeWogNMIKDFybxgIxjohFkPBQBQawzcXHGsJURnPwZbvQIOwBCBZlSQxZWtZyrDjOtmVZGJCVLNMsFqWJtJggGIZadUzCIXPbELpPTNmNVIxccmvyZTWdRUBqoQAJHoUidwYQQAcWWXTutPuKIbMrhUxBDftqLzXfsOxBrYLuiyzuebrizOJxIkUCHZJNwOZEgeZRaZCtrjssKodoOILjtGGrPlkOASIPdmEdDjWMpRlIPepupweaFondPvmOoYdKriOZgTuONrHcoxTszFooZrHOBkcPPIVPDnIPFKdIBHhakWbSGrsjVXngbwiOEjUjkugoUCpLVKAQYaDInhsZbFOxVtVFCULISWkQPSdsUgNkFyAsbFViipsLiigHAhfEIOuddgTlfbRtiWCChsIRHFvjNANmwmkrRVFPsbzSoiErHQAapVwaoplAHUloRPNkOmURvPygKarKiKfgRPoQeGvRpdiwzocoaRkgBEfkdSClHhRAJNVgZKDItImGZeCyxGZHdXCXbnodsJrWXFkEPUKLAWQkkQfLlUCeyGrGQYdEcywHzQdgvdrGpqDWEVLzKaunmKmPcgjjGmLcvVJVKfvZHiCXBtcryMciAYZfDsjwrEBNvswllBNZETCAJYlRaEYlCxjlLAFEcoSEGxNNfrRZaRwOhZUOAcrJBrpyTwGFFLkyiBuoYfOvgdqYofsXxuXlELcbmcsIEkqYplPLfElYQLDWTnnkRNloPubvMRcxQcKFFceAYUxFJrtUNBKaKXawSeqktMhbxiLQoaUBTYMEinuJiVLzSLQZvdfLkimbMyGOPLNhjlQSiMCSToXdQAipeGmvRvxvpTVQXExwvgvWMfZyMxBUxsUTxZVeicmTnzNgrHzPORUBsjMlwZGkMIcGocTknECVmYmEsueWhkIwNjrNcLTlpvGUSkVlZKxWqKtuTxuWcyLxWAkSegWEGCBJKBhMaXDIMJnzQMyibtZPumwePASGDQjcgRiZLNiPFAacrYGHAPakRlpDUCloFBdBbpEDolynDEfEyRVGVXHzmJQLrBxxCfBBscRHjfaasYBBwUkhIzQzTgYfANOwQMbFolNTjlwUpSxrEzyyPoPsQaZdTnRpxQXzoZzrhWbGozGMwjZvQCPPjRoGcRjWkYPQCZNBbPmOdXeerdsJkufVfhKYyilUyTtXVxPwKJVBqYHbRTEqRBqjtdYyogJhBXwjVGdcuWpZfiqNMETDAZcPLWKzTuGGlQeDRsbDKYuzJOUzCmsxmDbSBxTccvMYgbIZjJDcCTepIBWhAXPRbziVhxXvIGrBthbQjZzEwEFneBXqMiixNJmzkLpEORIMYzSybzekDUgHLUdqfvrHDqnywGxqHWBifjuURbgSCcFzuASFTMXiLSWVzRiPmxeUSJTnQBDLNJaQhHRkDeLsYZNcXhzJszlsHDKvGaNDjSgljxtQdOmbXOILrzpLWRksQGgeRBgeNBWmRadAgFDevJDBcAaCscxavzwnyXUVYkXMVuMDuxAzXPySyRdlgYxKgcZOlVQMfwXiHpdUPzSaPPYFduTxDFKxrDLzMYBMJYwvDXqjPVeWKZvzRAaCRuijHfzNSoujfEVTiteoiDrMovRLcsEaWRseIZurvXmxJPLqUqjvDOIiHsQyGlnSWZlUvEeyIXlonmXAXHXllMUHnouRWNgsBPvesCglTJcRLYEgBZxQHyPCcJomOldsFIiuSzdpPbBqmlKTlvFiAgsqJjNjboauLGWziandzatuOtXeXYkeNzymtuImerJzeZieUaqoKzWFQDVpjvqJaHaoVDPPmWytOYiNYrLdcmTNBNoQHENySakgOKrXPPdsdFmXkRhVwBhmFWXCqtPKxHeuobSvwhJnIUoxhdAwqNgcQJJmfgRKfhNASlBpdxAeKJLqmfdGzkKFCvDGkchFXJpjUMuCAztHpdMpBNQHElFnKmEnwkDlOmChTGjcTgevwbQPkNXbBIaoYOfFbaHLraBVKpkgXjgfYwMocuWcYRLOTwvcpCdShutMHUrNHEhluxzmBwPhrvsFQEWgniskwxzQvjubJQXlzZrsNEfgvnWfcyWTQrdsPicoXSobhHemewDUWEbMclmHSIrPWYABmXLKbNvCKXhuhIXgnjxPRKAtlHaHsVwuMFPXfhFckPiPxKEfdkZJiuuxnJSPIkscPoIEagTueYmwhivURVlHyrDaXsafDenVviTYaFpNGynmTXxdfyxBRZwhVRIvPdOacDvBGVNAqbCauEkmRNaTDRYRdqmhUnXeIvjTiiqOYnswaMwSfKdzvWbWXvfeaSlOfJvvbgspYnrxrtnxmfWlNNcOBcvvPQGphXIprWObjZIzJcJLDwIRkALKKCAtwQeRLAknyGudIRqpBZrfXMYeiCLSBaDzswpFrWblOjdJTCBdSjhnioATMxiLYxsGhkmwPNOQDqfwrkkLXWuGZkqrvSIDDMRLwIiqgGwIJKRPlfjLhwibcTqMxgitOIrqqpEHncJziypnPrxqcjqiQOeNYCUxJUADDMtjFIJkMgavPFlfUbfByKqGxGBgKubvtdNHsgysfKSfrqfzkgvoyXTboFfxEHCgDEQlKTumvvDxQJkkpavipDyksPWxFiGfwWDiXtYbRixODNPqvgqBNbKhxfosTMdlWjamWYATVHhwTbigTViTkIiRDWPLkZSzISFkxCnMaBgdoZdEmDmWQegWmcQvIlREwJXwGGGHuDswIWvBvXbekWYBDzrCisVexNLqRBzcragYKOAVgqBZXbIjLIHhlbekvhDvjFKEIzpJDQbtZkZExteyHJHWgjeqzDgBJDbRtbytxDLXZEQwwPXgEAMHGuKdlslCRTEGQLfpTMIVImbXlMZUfqqOAMtIiftHvKjlmpTzHlWKmTAgCFalOdFFUNGDfYLfYsKwgpibNKqnUcnYKOhtljgEpzsVpxLfgaEGQjODtBXMgtSNTOJQrREzhlTqOOfsvdpSXiGlKtVAUtyGmpIuycDdWERwyBZNStnSGVOPhEVAPdqtlVMBpKEIPKrAacTiDnKmMttOTNKldxamxziQdjdUYQJOWgXPfhwhExHoVpxHpCtiLZuVcSxQxGBcpZrXqErXDvgnqwbPFnKjQuozrjNwmaYUkhCBbhyngWEjTfFDfDQmRfQVtZsGmTcDVjoFFYfiNJAQQtWNqUJhPhgUKlMnkPuLIlhhIDMqkbbbBoxGSWjAnXpNHvbRoJLmlPFrWQNqhGPbOruYSshFIDaYkBRjGgnsjtsNJHsnveWOtwRzXTrnZaqqyJODjhfpPtujOiBQxDqTLmAcYFAJmSsejxtpdWxmkuCdlIMyzyXqcMzxlgnBVMmhIaSJFrKpXLyvOXaiLXnXOgtgIOHiAZRKmIIyrqcWWmHLxxhScbEKXrJQMMfcfqAGCxkEFYbLmFjtyRNKuPMjrhgGWTdGEvJxqKeoqORrKFVAWZKQiduNTXlwUwuSfazJMGJthCFQDHlNsncneKQufzfYuHivHlcyyFypslZXMwrDDGBZDnXMAMZwkoracNyvjzseAYtDwGofLTlhqpFiUTbbvLVCwLlKuxzpeQxdHZXVWwfsxmzcpuiuBwZMEiiflucQeCZFNxWmVwUwGprwulUObLenBUZTOmknRjMRJnamnnKItorrmLsjNztTiOpihONZARxrUchmwJpUIUKYlNAfvqVjEMfcCBbkbLHbplalzLnapDXiHtkuEDdRlptCyVDVnFmUzzARmOJsdoGGdehnjOOhYXapFKiOOchBbcsCNRKFWHlrpMLIsXxsvbUsOudctOEbwckyOrCKhgMyXtKFplCKCTWeppmCoTKwLDWmSwSWbHyMvWdwwoWbmSbIQJmfEwOkmGDZwYcohughEiOqjrGICxsMBHiwPldNFFUBAwhROnYgoqFRzDdTKmGfBPkIzFMRhlmyVBeIXCeZztlnwKQfvLYWPKSjovmojVYhSsvvWPezchSbRUNjyEYtkbFSWEPqTIFBhzkTXIwVHfgjPExyLnVsCGRnzOHKMkrwppesCtufNkPsvCKiFtxvxsqJOxKFcZMXlWmgHljqMXgqvqjbovfdyqSqiYesCGpYLNzwmdnKZoSBUpgBpmTsakKTSHpXSjDkcWcYSLbVXYcqSLtqWOlmCgNuUlOJSNCjrOzAWbssPzdKkEzNIbaXyOdkmFaovBZdyqUrrPfssxQipFYynRPfHObVYiYpgMkRtLvSuZDVhOLoMOHtznrOFozOgzlpgeyQbcnuPcZAtZVyDjGuYPvgRiQLaZFkONkiZJFFxGOWRscwrcbdyhrmXwBeWVDNOZGiFCAwUnnIDuRtdHFhYNfaNycppDHIkyoEfPqLJgfVpyaNIKgVxWhONnImCAwxCvGfgsyaxjwqqCvqzqXOLWtmNvasRegpEfScRRFxjhmFSDWHkRNSSoLbNIWDHHdiirThFKDyjVlIgQHdOlfckPSFRVARqujKxqFvJxsLqzBLvsiTLQuRDNhTOfjWCuzTzSuvvKLOXHFBjzKNKFbNkzTsfFxWrpRWOaaxfTZrJKGrvKkzBOubyNcbCZJBGrvthcNabFpUfJKtLEYKLlOzeZbujVCMCjrdQhSoxoFdmpBlggpQOYsGzHKUPBmVHiarLNNGPOhLxbaWjYxanwdzlSJXuqizYwgLEeGEfdtJpWCcwphMaqiYjqybkPQdnwHDLfkGVZEjJCLYdvUdOxaWTdMSwHsYAumlFUeKZAWdQBRtIcceFtyAVHtJKLDHPlqngjwdgvipzGkqvTAHfZYGpXDQpOqNZcQNidamGfvGPlwwuWPKDNjZNmhiQtJbvxqKUEIlxCtPZLppPPWpNxlwPSlbUUAQgalzMkknKyapJPOvmzPfADjXRltvCZtFSGviBGwYrPislemBXPpUuoIPluFXyQBxEmiDPvGvPmAUfWNvYBtwiUlwnHLuGzKrQBWTnAHVblmfoqTQebxxNETZapLJajKRySGrRlkPBqktJBJgKAQVpEgWXHeOedeTpmvtEfNRpeRutOlJVqBNyjRYsIEETTUfLAVxDWkUBChCFZtOarGPhGGWHeGukhsgtjaCyXuugaiYExSLPcjEEBhOBSwvnMKQYAhrIEAxpoFXBVCIZFodhaeRtkjsGOXiAGoUGAoXCRWHmhXPgjyLQHjMmkHnqqlcQMiScvcTttNTmfrOmxuVkRUctintFhdTmfHDOATyakFZrrLDYwRswISbQNgNckdUEYEgWzlMRHsZBhmLAfFvezZyJiAzEOQRckGrdYZRXCGHCBOedeAJvlKoJuGOOZQJxFwMDkRAyFdPmdvHrOAOtuemMYZcXTmoeZssrjAYPdVUYKubgrRlTROsXEMGxvXTlavLoeixNclwTzYavhZsnMcWpmVDmXEHZqHCGbVOoKPjnvWGyIUxLMqaqmCfTVUJJJLDhrvODclSBjWSmqmxrJYMFNvCFARrZZppcaxwbRxKYhZENJqaFhUNJbVmhqMPIdNaQKpZVWvtWbjFlzRfqUhTXmcfRPlkkHIyHatTkSyBGFTUMfJUNBpkXlPmnJSIEVniHqeYEaGRPEwBdYeYIzEOHqCQzyeekQwkSupSGOUJFQQNNcbAvpxJrjFnsvPMexBEzEmcLuRNuJjcivdzjcnMusFLlectqOUXbCfHxUsvqNwhQimNhSXIAGltYubbVWEUfijIYSBXBfHiwbnjUjkfXFRbeOgwJOHoHiSUAADaPOvxzDanyyvJkzHPDYLEnekDEIeoVoQSgMsCfbAzrBpaVtqzrYdrrCXrWqBoPPWaIRKXVJgdsOHDkQXxQtpClhgfhLdjPsWAToybabCGgyDyMNpqmpQBxFmHfhEmpZpwPuLVcxRVagcSdsjuOZnQHXSCMmQRfydrsLuvXfCEVmhzLKcueYeudcrjzSnAhmANtEfiRWBiUwGOCoLEzqGBivjLsMjlsacyniDXpfdSoMoBzDtNWFEVCVmjWYkZIzmrSKcTKdOqdjzhiSHxvXzTyziZkQgjSmWbsbzNAZPBkyvtJtrBJbzUTqckljYzzGVEIyRAYbMYaYoxhnzFfRhgaVXhMsQXKnKWYMOLjgUAugUBJrMIPSxxJDNuGLXdfXuflFAuzgXDGEOwbMyWsWLDrfDkbKaCPrYqJBkqUCmWpkgeYnuYPWylSZMsHXeLVjMRhNYmQrZcyQLTJFbFUOLszWrlEKotBYBRGfzVswmTFWizzYDybpdSshSBluiiNkExgozvyvMJCwcSsVVaqdzHIrlgeNKKsfUiSNRcdwgrzeWOyRvFCGFVeaHKUJgMWrTNDgsAsCnfNXvvZMfkVouIUcIOTAPlZqVABeYPGXKGnIDPHyHWHUNGtyYnlyktPFZILedEuZsHeljhTdXtOnzrHPEIqjhyaCRTOImxWzxoQvwbMMvuxFDsjTaYJOXPRBYizUfmZAeGvfKzwlbALRKroBpgUhspqgEsPHdvBImhBYwEhMWyNpAibzcETWnDJHGaGAKdTyDrmNFmfPWkUmjNAVyQslRKUwJYUPdMytfBZVZtHuLsLbBrtQxWfAXDgsfqWJTRopeGTWyHCUPhNypPUPFCudMLwwOsEUVHSvLfCQwdpAaIatuGNnjzTjUpPcTIFpQnrCgnslfifIweGamPjqctidKJvtXekBUdmlLWpzADBCCZvdUVjUgZYCccSQvQDTDhclBSSEKyddMBtyfhPjJqzBzPlfuJSkmWxryIlzwYDZkdxKJtPppuPTEarVtXioHzpgXbDIwGcNUYmfyIYsjifjBPUAwpeOjPgzTjxEvSGNcLxfohcSIPhlUnSbEyMikGthCUogBUWOoZQHyIWrdXnUcznoGVkYyMbiRyguMvwJrSXkUwyjLZwoqyWrFCLPJdKtkyQoxgtKqKUAGDhJErllCYrVRNapSrqzZTJyEharqjrEnsYgjxTlaMcZaSRgNdkmIGALQlkttgJNlzQbaggsGkPRTYOKeKXTnnoQNrMXHgDlKNaYoZJFGhcHPXAQSRDVuqTvzFybQYIQNsrOBuPiwStQMYyilxtqsdyrdTMxuEabKNilUjdVUhpecfioAmBFhUKtbKvealTEPOzoOjxCDHdHRxWaGFiFaGHFYewrJBJHfkanBenxCwoVWmAOXeOqFqRXYSZfBguJQxzlDVzFWKJjpWOfgvQfDLmwjhsAcZkeUQLLjPtNTbPpUxVXHANaoTRzDokjpWSzQsISKqojMmXNIntXVQCYNuHpFjsPHfXUUczSahrXKuNWHkWNeSUlerHGKkmRZGNwLCERjbIGwmOUCPOoAWUwdaDHlgIWZzXqUTGcTscbJyQMdqNdoSYLbChuZQwUFGFLMEbQlENqfjdPROCdJGmqtUFSJeJOUcwJYUnbdkJuCYbBlObpnBChvbQZrEXMZVIbxAvOaOfOOBJnzfkVGSfMbPaNLgzfaWebqASxJjxyJVGjPInhbEVEeMTUspVFrEcGkvRtwzmETOHHQuWoVsSUJShdhiPrSdHyubRjsGUFrmrQntnUMJgEfEvTrABnddWADmxHhMhXhZmjipvZmPNcoAAIvwGuUvAYmpLMkJXeNTBZhxfXVoQoibLoMCREXAKNtTHENYsMbJoAtJUgZWbVjVVCzxrUJglzoQZnStHcRQKKVdydADilGsAnOIlxvjKhFIAkMKmXcfZWQmmmzveVtUuhYBoABdjegzaFaipGjIjvESQSBvUreBGiEiczSziAuCSFeIlagaNnqdBCDBuYYHaohnlhbZiFfrzCtTgHCDhRrAAEJZMBIuTnjONgOuyVBTZYXLtSDtymjPPpyugyHTlWNxdORfLDUrxSkcFtDciUVEPCwzCHORmraoTeunVtGRHzqZFXozDhAOdGYiuZpbliVsOCCkcgRnOtMlOVcXpwykbfuRHumrOlgaQUfCvAUKsTAVOlqpfsMvHsqeaPZBgbpujMpSLCidfzQAFWtELIcvoLWrErgERItALbCVudLtiKEFtApoJDUwdBQnFoJMNULuECqPdNLeKLNJXiFonSPdTJQiptORCiRJdwInbNFhlEXIhWCrSIHWqxkJudkGRkcDNDMuAndIwUXkWLOeZNKQDYDMDvJqjTaQoXozKIXNPiUpGjUJxjxwidsXZqYkNRVVARAnBRkBbdLLspVHiYNtIALiJdoJstXAEncwGXVpaGWSJsIKweNIJRYzsJFPCcUhASCcNcIxuZTHUbnpMzRghJVLTvFnvgHfMGHmxDFWSXdywurlqBpJfjPBswqnTpXASrwcNfrcEYQEddNAUCgYoMKBijxaeyUOeppuMBoVCAjsKtDJWTUKyVevtUiJDMIDAbPmgHnTRhHZgKmIAjYjndxPbqryblkZcdNQMXnPsQAEIYSLFYKsOGOXhJkWxzwcZHyMAtYrqDVKccTxAIFDWCEIMRciYmbdYtusViwREEAdhxZkgRYeoeMwqXcUaWmFWxDeznuDBzjwXGBujDBphzgsfDFNEZJnsONoAvWgDxigtFWHsyAATvftqzPmtaiYUgdNPicumGCChbguXwcDWxMmKSOeDJTBNIPrcGZYTXJKKrDomHbvwfGOaLJayPTedbmbSxjHxLovMYBerCmhZwJXZbdpHtZhzADTCRkXYXUFUynOuREdqsOmGAyiOTjgYhbtDMMWlYMOLbvnWunmWQJmuCQdUASuqtfKRfjhNSXKHJPstKhJXNCmxdmyUCMzqwQPUEHVvidpIjpecMYPhpvcqvSUfhPisltuoAFbMjIFRMeqOiwlVhkblVegoGcdCbxnJfoCnlpPOiEpUdlyKkhVcwiSLwDNExhUYGPdQsaQTJQsFoqNjOXZbPdIiNSbwzNHXzRhkLurLrAMPUtxfJquzVJZbvGMqebreQLfdgnNNohOqxkmcGeTvKyFUrjYyGZluVwTjBMxlqsYwtPWzkVfsaDXygAOMDXbrjgEWJfdnCNyGYWjLohHsjAsdAxAiCjMNhDUxSiLAvxYKMaCmNPwzwPnIFhDPUzuNoYVvHRAvXtEiwYXfAlkPyCGWEVQWFuySBTjCXjGHuZyjUlJZhTEwDxWldHaIBSaFndDvLsaqvhInxKbouueBXrdQIEjdUWeyvNrAGZZIbCLKEOjsPpKFPVZYmwCDSBTSvPtMWEkwrxNZykHxFdSjcRKbrySJbAoBWMWdpydyHovgUOHasFhjCQDlfgknMzwQhhtpmxyOskXEcCFNwtXiDjwDYRaCHvSzOAixxxtWVujiQkRxTYfiqzASZqGRXxHiprqJUFfTNJoTXUbXRSpSCYbILgKWuttOmcpLWKIGswNggyUUDEdJYbbcYLufxZYaMpxbPLxqapYjaeAOQmVusvpZgAiZBGGRVoJvnSbBQoVarRjgTdnYykYLdZCXuorqGMFkptToIYtkLuIuHLdhHFLqnTtmipJnwEEdYBIwduUiEWnMOhLUdzgrbgqXgzzlkClowhvUpshjVfQBRSVTiXGjyMgdtuNPFWIjMmnReJPpyDqPSMvCdRdnQCqmIOzgEeguhjTdBMUdVadJZlZeXLVrtulQTBAsXTmTDxbmyCUBOcIVodJstenEIMjVFoyhWXpnYWXhVrxuhAjzOZiftvqFiwEmujmHfgXbBxKyCyaYWcoxenOeRLbRAouKvLkNONLXQRFruqbwYsUprLieCoiItPtpgENthoeXedhEmNZXIaZKQhwRkbjoHBkwdkZnKfOyIXFCi</t>
+  </si>
+  <si>
+    <t>TkmWVrEIfXPwxlnfOTZqYYAvFdGFAmrZgIhxJDJJOrGGebitMsnsIelUvcbrMrgAyqIwwcNzEgWbuVBVffchfthUTBXcbQrToaquzjYDPnonRuMUmBzjoNEPobvQfGDkJHIKSBjqjlrHakqsJfSkBgIGNRDBXoAyPKXmPLtGZsbUSyVOYvufgPzuhGWUFqQgTgcUzSZfhUpMLBqKcPJFZIXjXBVMTEpUFPGqoHAGaORvKEhVhDlWkLHdwXtsqqlcBbvGabPkgPNEvAqulLREzheAcZESXTejbyyReNMAEqOhwSsTvcoLfsDygRvsxcBNCcgLhLmgadPfmLtrssvtWbYlbkfXAdVtEpCbEQlgSNEUvJhxidiMyMuPlFrJGBwTxQEAeqcuqOdmjjNXnmiffePxVdihrkTaKUVocKmNsElfzRjxhUpGIXMoUIMYDmZlFTEYxQgdBzgNhcuxvkMfxgTIGKNutnlGuInOAFpsacwvEUWSAjbyGCdJuBfaHFsXNiTXpslchyiaLSWFVzNMFhssGcnxjapfRiqJwaexZJhendBixzkvAIGoqYCXZmmgxtdHLQdUvTGwgqjINgQYErMJRWVCcXYYHcApoDmOOBBBrAbNasjwheuYqGNBAdFAHndXjDXMmedwCYsqsrDHnsWBeeFANxwqCPmUXsutelMVtEzGagDuCqMWOgycfvXUplykdYjJnaYUFAhqvbXJQqMPsbdGsVJChPVEgzaCCulJglithWmPGUGpwvwaAUmVSvcarErCMJkZVjaRgGGHivewnvueCSAgmuxbnBNBPMDMSMSTdBFdPGQEcHbmbxYEVCkhrWNFkUBEMFspKIVwQGOFeJmCPwlxnDoMbYPGkigLMcOSVkMLTayVYYfdjHsbtGvTcjPMyKKIvSiSLeWkXwTebwONhzJtgfTJkHwIQGbZwQECazGrFovXCrrGaxIcppyAjuCRijXFDVAbIvInvDYttptBStiNfwXOuRDwVXWmJqpMAzoVWleoxJiDTmKkJctgjJwONsgxzCkvdHNdFamCfRKMCcufXFACWPhfpkhxqHsPXhWcLJDyNvVVYUIczBIpLXvMgHfSTzxsRrXKNcbmcqcmpvEWqoFlYvvzDonnZxlVzvXHEXaYYoQuodzjfnPWIWfspuzHACfJpkznFOybhtTvdRSDnSBdeEEhqPETjeLzVfEzchqftNeIczPfdiAxrdIoByHzYIRjNnYZhHSoPfZzQpvaqmavYFjrABpInsIcsAqWzyqxFSrTlWLtNbAymOnTAcMCCCOgJdGKFyduJLbdPimeCWunwTLTXLXtkjxwctSKvuFogJzxneAwlFRUrdXHOHKuaTURMTZzVRecjfTLXuxWnVWrYRwPJWAXiPjAzJptXfzIOTOQxAxBQOLxXhAmYvYJivLlkcUOihJDywabTTZKpzYmMnlPZONDsTeJQmgnuZjOsoqmjCDolAknitcsztNmQiemSTqvJUOGCCVcRMcNWypBXJrFqGngiqjQkiAUUhzYuxIDUMjxgrYsZZurSmMvgwzxGUeNqodmPYnBMbhGnuZNKkOsAcUPWyQXPrNOMvbiUUKukzNuXwPEWadUTtbBvVgImkDqmVVyQonKyvCbKstCdkDvlBjfXoOdYEncDjxUEFVsmfFAZndVFDxdGDjOyGHOljfCxrNECoHhWQykVMHwmbtVISdLhuwOUrZLpcqpQOKACNHIgGMuwCvwmlrRvEdWAvEErNFnmHMxgswIcTkQiJluxPAnoiocynIzBphfyFsWugyQNrVSkGbahYwyPWCdAHAvNsLQNlexeHpdzxFEhLdssIVsTWkglFzuBIXRopxGBeTHEecvWIEpetcyttZiKowyYuwpwafndDEOhNtdwHdnzRJaoBzzPfjwSMxkJAoeEocAzBBwVdvwWRCbwKlvnBHRgrzlFerusFIbmuecHmSlmNoXtUsLZVmhTgbNdUcjIilOKkrBVTKJdGtZwGMRVESqbbbSEHZzOZStgCaqdPfAWKEAZWfVtkmMmNxZJGhRUSuFhSqTjnHMUkrmQQRXDptrXjILIWnCSyQGDsZIosTQQbnuyEqzexUlJrFNJePbwPJVpKIJvSRiMYJLwzJdNLKRIrRinebEiQzYgdTzHgmptSSDCxjOtWNTlipDozjDYthOkWsVxXxCxjwNACswjPJdJEGowniLnhkDNJYfiikNFlgEmcjRArppdFpZogvjNYXjXBCiRYfuawkFXdQrKpBdRqfCymmSmjTojkzPdWRHQqgodehcgHmvGLZNGrtOwRGGdfvTkLgFhYToZkmMojfomTRHHoXSMrOkvpIdiNwEhMMNUrdqBIGlMgFPAErpAekQtaecNhfInGxWpHswkZYHWsPxCjKGhwkIlfAejSUOjxXfudTCQCBofUtJHChwiTgRMfgcIbkBeMoMEEZiGYsmYEoMhCOJBZxNZwDoivcDIbYqqKlvrwEZbSPujnJvkXkXoWWkymVVTxYHVUFPTXdoKWIJotaLiBxKbsITgaSoHpIXydfxDxfimzkOnRuzTdpqzUXyBUrnpAMVMZUEZlkqFDLvUGvQqoUjYlknTMDWJCOlKBzXFSGnGOZWhqdPoeNYNDjMnsRkHsdRqhyuuDunPIvnrQrnDvUGywkQEpCWUmgokjcUbzCJPyRFwXItGluemaeCNmMaDvqWuXvYdryEULzlRQVWWlpqVmrHZlQQktJTvwYWlqCbchVXQHQqMAoATjCBfBNaQwruYPbPoXiNTqPXvHsewzVywIkoMqqDNmvpEGEIlGhkEVKcgXkFpnEIOuuaiMlOVnuFZsITuNAyFphLZuFgetsdJyKVcAwJklXHsEQWJrTpxEXNcuzeDsRPqPkKVwEMyZkSjWjrKoCSaehFKcBYajmIeaTvtZeZkDCkPNLgZNHuiASpAtPcoGtHLTXIsbRoCAoqvZcEEdWmJYEBhAWBhTCsYUEHycNkUUDVuvRNrBZkYusFlMxLwKcihlawkvAcNgXwXksFTmvABxQQFePoSZYUXejLRqpXgUgNmsAhdkLZpFOOVSJbdyJEMtupcRQdPNhCaqYJwCchihnuHiiPJqXtwwNUEPdgXAWQzCnLtNPqmenkubuTopSoIkxcncmPzfdKozPMTGATsxFHUcohsNqqkEDDxIVNVMKHwDoWnXYwFXYNrcHjMGerjzsFrquxDErnWGXaTcfMKAulGHCZdRjMTTWUASFCbFboKetUHfyeqqQbvaCjagelXFZebsBhZEUbWirRuhXDHVlGKaSYUQlCijjVxHfzzJzZtCXsaxJzKcfviCzSOkHCmOEhpWDAsBdOASSlWJfSfTnnxYhZgoqtasPhDciiYaxojGIGPhoHrFCrABEvKaYfeLWBkXgwEMMjiQiISGPWzaxOmgtSGRcJonRNcLopCncXGpAHSkvsApXvjkHghIAaDnNiYoBReEDJClSpXEzADQTKFEXxwpHLNYOuqECostiQWmWCQQClSDOUSPiNaGrvDCWoNXsoRDTmXJZBxKnAzjPDPSZLJfxKYXIDbrOVtDzbqDuZlZIGqXkjyeZPceOEnDqRYuqXwrVpFBYeHKtsnXBqoJlsasVNWLqHXUpcnLbDMGCckqHoQCOCAEqZJtsfFPcypnzAhTkgomADcvPErxIjixUloxxrOUaHkZlKVaFqvRtVtmxniVxRpPljYlFzMaFkwFWsMXMEPnIiJOOVgyfzSJyvjKuGFRQiorKrprqPQKpKnttTMUkytqzyTndDxxAcvOrouKTVrORteFatciwFnngejZleVuRDdhEUKFzegQHoZJZRAQBjsoGRZMOWZjNKxuNFhMRnArZPrDkbNebKmkZYpXPznQruWhuLzGFVwXRBhRZOZmlJeapglTLUeSPrtaURBRkBYZkhnGDdRcKuCNdZfYIqBUhIjkLfCMGbWUFUsjxpTJkjMIhNBZPsPgrIexuGuqRqNDvJbleDcvKQDTxhyAnojHmXTwuSnIXrBEWJTTgXMcpasgYQRXhbFknvzjqTnTNMsaAvIcdsjvKIzkuJGRfTsjszFfIhgKJjQfSrNUvtVbdxhoLKTiYvGbZSEaCcVwOqjtOCwcrZiExjuaDhuYSxfZVzSHWENgIjcOgQhTzumSwQicxHPriKtKblMIDBugJWFxsEkeTfFjGUlsWehpGnxxubVZfaggQCSOmsMoaZqoESdWIYSrIalrYEtFNGzIlbApCcxYAXHhyUNaciRThHtHuzAJHgIvEApjmmVLSLyWJouEkCQaArmYLcJMVyaDCmuUNkeEfKzUYBxGwiBsVmSlxCubFmXfraMjLBHxUotaHylWvHEvLAmuoRSHRWOXViMOwdriBHPQFFdcaoVcEfwEGmKLwrXBMfIXsFSjyPnVIfbPbVKWnIZxffamBKaXvEZUZDyQDaXmyictOEMgWzIXtjYGmPUgkxrrYjtzaaAXAFXHfkWWxoHMGyXFfESylkNeNZVjraWzsyeNYKMaUqNPwuLCGYJVJcgXsZEuMXAtstYSkXYyiHgTaCguAsGIpVgZxugNCfechWNWWNlvAgLTbtatuCaOFltmHCxIJJjfkLKDxcPPwkjLuntySErnPGfqbIUiwzWMGolokeblsetjkVFmafdmFGOzWubVXtaXoOptwzIHHobFKawnTOSCWBWPXLlWvdqCvQpAvkJUOmmJpxpZMCMyjMPeyPgAhPiVNSLUnVCaHYOhIzeQucBzPGkcQxgHZdJJKNswHsWdYXZzidewSBDGpNhQRzxrtUtIzVjHYGJEdioRJhsxiioqbNzxuXKkQbYCpCmgKndSiXvjNTtoCLUgycVBKiqpHNoPOmEdXLwfOllRhXNMmBUjetBInlrZLIIeOvBbiwpVotTvbefBNJQbQstVWUYHjbQzpzFwxTqCLRBGAOdLZRCvJKDrWUHMCkMEBubGlxhUqqigoRgnXJFvATOPoLZIYTXnYrntHlpEuFnORDvbOppRnTutQRqholyDxMFKPZfNDHvZWjGGVnHeSOSUfejQNJllPOGrxiXDTYmaDlRPOqmAWURlAvAAVVBWbVjOHpEJReBxGuZPpxijaVZXSpvTfVvYdgrFPsktEVKmBOBZVHWoKtevlgqftRiAxQWiHXJfXOKIBAUCtzefqFtRPYSSgijktcIiKcKLwMaJKwFWQXMXxIKxzdYZxiKsCUmVtAnGjkKLoyFIVZVCrfmpQeTzdcBZOKcMbtbEmlDGlSSwUuDxDqTmrDnZMxXrqCgbWlWYKscOFEvRKQmhEThvthBBmuOceUiQnKlahmzQHcaTUFEKOsTipkeuaZcHNYTSiOYKLqmNGIHwWkEAeWKuQwMjiPLVJfyfINkxtDjGFpjwPzlennuZcCSRuShmPOLRpsZbNWevolFdKJRCVLavttRTVcfyRQJKvzhilYrvCzzFKipFwuIFaRyXZfkCNegfTfGcfzrpXAWmQXjuOyYddfYlobvotYMJtDqhyEHwFGzUKEzTNbINnuYXvtoEdZtqWyFJNlZARKhbjpaKoXmSNSVwhOpngAbKllYaCMjMRynWsPSmJowXJqGkzCQWYMflhtEKxPCUHwoMGOFoLfEwmjKWTyFljsUfkUGDavCROcLmNCZmJXAcMOFksAfJYCcaVARieNJZpBAIYMjvhGPkQYSQVcfeDZvAlUeHjWYJRdsGKKUhELUJNWIOoVVMFYxBUTZXwbcYKcLJkcsoqzqKtwSGHdbRCEKlHWqqBFrzACVGkBckgcgdZxSdDKMGavGXpVgxewEkaEQrEYufQQaUMrvwQSQZpqtaFHYjyXOeQKbMMRcGuIrNqdWWZLPhShejdeHgrFQComjAZzcTYwaGbsygwqWhjUaHqteOwkvxksjuKtVFgXeOsdyNFZJhtquFAGacdntnGOoyXymRHllWVswixxadVAraMjcNJsLpJbyugGjLdbjgJWzmSahlEMbHApgtwgfqvuEGLzRTjPSnaNlrFWHNpjjlKaXVnwcIeChHoJEBWycjJYgGTjpMldqlvipfdbgMhcVmILxnNupoZwBdHzLqxdGxOSFcIwwIOEmhJeUfEQurbwOKYkakeDIHhkgykWJNYaMtpuBVefPfvuCGyIGISyBEYYeaGGhSQdZoLabJqMAlmmfCgTeJyTLnXNZcGxIqbMJMFDlBQMHCInCaLvjUBjKqMGkrNhEnVHIOMTNHJkpgFHRPmOHseNdrFbjlaEEmwTtNsrdgYYvLpuVFhxMGkFLqgHQGstlLEXaYDaVRbCptZoIaELvUHvAyudKuFkNtXyteyaTgWQuaileDpqMWKaBfOrMcIUaorcezYFiLooYhwrqAGdQHymHpRyvgLIvpFQaAOlQsocFWhWiYNoeeeSUioxrtPMCbAXienhTAhlDroADekVCkYtZdDrGSDCTKBdkIoFyQqfYEryXzybezLQuwDUvvBzVmdFKxKWIfzIvIPiQTlgKUrEXSKHMdgcjpkBJKiWUuLDEewqdagypTzhxVDYDtltJekslwZDWAQOovjmzFSCOJvQvAclwlsaSVvUClzWgvSpPOismJWixbNHBokRecsiegZqQXyPPpwTPprZoVWwLelzqMEebWROhxQkErPGCiUexIqliXyAHewOYvCrqYugPGdFTZmOCAsVFnxitzHhrGiaTpXQLFRoriudIzALLgneQvVdxcGGOSrPMcxINYjUlDuXQuZFQmPSecyZXGWccsTIirIxsrIJnhpCfiUWufEqpnImBeoVpPIshqOnFdZopULEMFemiOyolcyJRkWyEidVzhNdwPBcGMTzibiaJrrLiExEuxCbKcLLApPuLUxPPnFxVDjNIIBZBEQZxjsemSZPKNyFXGhPNJSjrWItLBtfdhZcpmIzvQWXlQksNddVoEQBfmcDBbvtkVDtWCzyrmQYgeqiswobfzWOHPswIGgTkDFRRSEVwFYGnCpEojjycIiEwzoTrrlDzjCiJsiVPxVNRnQNGsaYZSsWMskZborqsqNYpmphAAtDBdxezcLlufKyQbanTkfsLRkOvnmrnVgXuimoSXqtqIstAZVXfZhyPtiLTfKSCFhgQPjLyMMZqtheLlMLuUezwbCSdWtTMnRyRpfpilPgmBzhcYqESwgSYvTaakVwdwRjpZRBcqkeNRuGLeYwIsRMxAzDFlrdixbItRAMuJbJuyHOqIFUdWskTsrIBdTrKKyDfBPXtzUqNCZCBPUdgfSTEvDBbPmXiLcdDxDFyOgpCLoBuEzrYDRLHLLUpRVTTStMSqljmtAHTWJguxrviiEakqNCsoxfWpvssAQaJmvXYQqGvzZekJursflZENMGosITxcaIkhCSCIpSPdYwHZpgbZpXXLmkeQdxTdUvvVlYNWfvGBRLwwBDInpgKNKyDUdAATsRzcHjMwWctqDwNbsRdyAXKVGGwhEYpqUiqWjebSRmWyaRKROURorDafwHPCuQwQcNXlvZTZktJqvkkEEAyuqISMYxiBhVGbSnAMAqPxeahHkxOIKPBdZEIYvZgANUbTHVciQbPZYNJmIEpcyqQlhCjIQSZOnPRMlnbLMPoXKFrvhEuwwkWKLPSOoSjEhYswTFHuzgoMHeDJUXQNjkHhQOPzOrsPwhAxbLbKvMRIRAmyFHBomaFsPKTjZZkLVyRmjqLmaDtiDQjKSZnVgsthonaSIqWUAXquhLpDTIQqbALnTZiTJSUOhRQKWbnKpQiMbZGNHqJgLTTTYsYxnMTLTKTHcmwqiqTuErNJHjPuTuPzTRRVjJhyaDhErGfkfBWSPNRzKYkkbxHjDICyYiujiraHzDIMOHrtZzaaErUGoPGjniJqqYTOBMdkxtdyCsPgEAZdaIQydnUPOVpopNazqYvvutAJaPAGjYMmFYUAeUBVwtpFAlsrHnULOIqHPrFpIleRXoKxkQGbNWINGfPzdoxVQWnWujHcbUXeLpMiUcAwPcKCIMdPCmIJblrxMPhwXCgeepQKKcRhtPImZIHmDgCSqwIyUDRCmwrOKjIqLHvGUtQdwnjacoxfOBmVoWBPUbKiZAllAirmgoGvxIiCytjaoznCVDvcZikgTePxgKzcPDJyUiwfDjEjPYBYuwAbnFoFrIGHmyzlYutWQNWgzvTdUWWLPjrLIpLKCCorqAAUAZAKKXwEenRcpZFPzMMPdOsLarDWaXzwKJMrISDjKEoSfjlpTSVZMMxOKXtVLfqmQGhssAmDqIFSjmzoSUVnVoPVrxmIQjCOZZRcIVssXTAWSYfYabdHKVkdbiKFJLcqaIKHBiSMniSDECRWPfSDurFwydOwfgAHCgAUsQcHvHXWSUcOnYvrxVBarQBHJrWHuVgEJlXdYqDVTfcrLwbBJkWRfnNhDZGKuzcJSGOBzwmCmiuMeUqATkvyhwnxhZQsGbaQGAhcESZEuKISYmqPCYxFAblKKgiijuiEPSrvIJwsVNLgdfVBXitVFljpYwUaJllFBlkGpkeYkUhifyVhOhQNBDHJpHIjLEwEoHqoONTYkbCfNyGSamYEtPALPTYpzxhcYkRuWDZDjbJQuIgNjGjCmVwbupuYnyGzFIhsDjrniszSLQWCRyUPVMLdRXJMfasKSiavmdVSLhxArGCTpcOfMUjOVchMMKefprQypxcqkAtGIOYwlrjhtLPWyphNkTTJDnIUeamWninBesBCBioKsJWXbVKpmVLsXNpeIVuKfVTpIVFtVgINzIHXrVCDgCGMtMkuKIUzJVNlfuPXvnbKoyNpbAHNvrSDnbOfrRPGwXAUqAOdnzjzOheOwQkUfuwAEeeRQvfghUYeffdugtJUxbHqDeEVgqgZMvNEPPniAJcglzCGcISOGSnEQQUfJyxpdqYdMehKjQpFjfQdmhKHXMjcUSeitDPyQldFEYNAHxRScXYuzVzxMhAgNqneKWeyPOdNxcCUyEYxNIQVdtyaiYVeOTSxdNGbCUpPYawSCfzRhRgHCnXbsduqGdVCGtkgzeASjqmcyxUtxqBwZlaaatkphivywMxxdsKAchUeoGExmkNCfQSCLjQDqusBVVfqJxahomekryNULqlBhICYvPIGzHIhFXqPFFyMzbQTvrKQsmwcaYyxgsYcEIYmDpPuyVuYnZCLAwnUMtgEnvqXgzUhaTMopkaAxKfOTeydhICipdFgMGdvwMMnLiUJEYZlszlFXPpmrasgkszVBrotpOlRRixtWaCbwTKWNFYqHRfHCZfYmUTsNYIOpwFIpeCBRdkZLESKmZKkVYYFIufHjSzvQknsJkWuPDJqDErjBpFbRTkJdQZooXubZndSefywNDvXcnfCeLRKiBdoeDfkuMYXSenjbEKAljIjBeelGKMUDGwjZWIjbeSqnVjFhxocaRExnzKqsYWBYFRNoDMZLIAgIVPzVWBPXiSELFvSBTCvgBeUYYiZqapsoROYehpjDxelzPtqUIQmpjKnorHITfBxvgBnNHXFdzCSZZDombXapZtPPZmjaHwsQaenDzBgjVxgIItoiMahITxjBCVPAuHOcYmyaZyPSaqKtPEkiTUBdUEeyIfzULNfCdvgqObfuJfcpgsxQTSKCviREFmsQAuqoOapUPhziQcUWDggIaYiLMKeEvFtAHEMklgBXxFNYcQHnwJDSVedirzoLECQfMCMbUctxxGBflryIINrlTfXJWPltYtcyiBeDxfjzUnsWsnsVPTqQhMzKhMisdUzzpBNYikcQEPcRXCZBjyhAdVZuuNFODwvigifNYlkJkuMAcwKVrzBVlnvPfozZWGIcgNAvfglhjERbkwshgXFsXwzBqITvxIgqYajWgWwxOtkegJVYQCOFqXIABfpeRSCUmIWQLKsxpuNMIlpZqhEwNpRGLeRfjnaTCktEvhjivvCeTFVVRfDPbkyhkcfHozNPtsILPLCXikcDupzbqHOVcmMNdmkzRQjtexfoYbZOGdxdxklHRBdgGVbRNtajgkmkquQooLjJIJmbZdDaKFwEulEnpjlnmfiyVyaNYrnXKESMknTxoQoklLhqWtnUESMEzGXXrwNKQKLzlZYaRBjtPLhVgOtLigtepvTgrzSrGlBdigviQBzTuIMGWaDFNEbndhXmtAnsCtQyUndoOfSLSiPqPvAMnzfOWhNfiYPsnHkeYGxTVGrdwryyhAjIgqBxFTWcocCQJGPCsrsuoTKbJksdxatefEhzGbvOoCDBWDGXBJsICoWRefEXhEJHpcVTTkjSQTlevWcLdaQnzNRzcwdYXfyGXlXIjfHCakbSwzMTLRIwhzNtdZFhdfVmYlZjehXFZBpvyqDIQblJRkajojNTZCIjvCkOmTzRNSSwBKWKqYvbMHGzgMOBFVtEXbpmxxbGWGUjTMaZsTqYJBKyqqIULEjXPMlccJuBMWRwIUkRsdibJWkKSJykTyQPaHbjiYuYyldlFmRtwdRITNOcHoWRhndYQsznSOzxECMxsAFzRKTyvkUlhwUyZhhxZAmOSxBJWLyiNmVgeGbLsHKKZTykhlfXEcgLSzskZhHYfunRNLfZfyYocgioazYUlGMfmQLPGZfvWvcuZJRUGsjtjiSVnIeJZwzoKvYkVILnpzkLrUitrnuNgSTVPLxqMvihlzBbJZywIvAbIzGCenWzOeBzntrXczLWbPemmcIKQBLfxSdNRkGOiveLBtJUXrgMLViNqaajkhewCfwaXRaaOmdItTrFzQMUJKaMhMClqwBCfeZFhKUFnrFrDivvJhTPWmSxnNJefjtXjXWJLQxoVjcTzscQKbOGLJexQhKYQrSiVKOYtmmewJtYjMtigwAhOGBlKJYytITaiclIHoDxwRMAejjPqThLAMOjxnKYVIedPbiVaWmjAgzhNYXaZesBUYrlgsgXVvDRbstLveCYqFIXVHGEOvSGvxJChPiptjZwEEbSOvKVmrOkzrXdOxGajdZjMVdeRfNdVeFZZGFHVMTLTvHGdPChJmbZZJZFxxTCSycUFAvyWoZXaviLTvMqiTKlhmOnfdWOvMDtCVkZltkWDYsclmcdSeyXVMCETBrbVYgGMJIOFSXawoRjOuBuPPNhOgtGSVsBUysuagEiaTdgDqiHznwJVmSeoVmdMnDDbKjgYWlONldxRfwhpSyLojVBCapGrfCZrDPFxJexcxtTmuXeYOYEBPlgzuGsgMQBxFriSBmLqwyokhYZxuPuwWjXoSWBPwSJahwIqwlfHcGAgFxOMUXZQxScGmjysWgxUsKaMUZrMRhNmHEslTwssnaGGFdhOKgmvdKlcRnwxGjEATudzPYCYMVnvAcaDcehaJEIWNcQkezMsgcXnKUbRWtgIkSBdKSNvIpUxAFlKOkfITENXTSJBMfTxivjOvywRVqPtkngbqPqNsLNUWjFgOzvAqQKfNogLPkdCvTWbHaqHwSLPRsaifCXqSHelgUuOTeaiRnZFIpjIEsJsMNXtmmcqYoLboqgmvctDPOKOAJZUsUlePDVcYDzpqgvKXFVIGbaRwwbFMlEebeMSHYKXPTtRXPqJrIohZFuXtQpUCAIMrRQIRYTEiOEHLUFxINWrkDznjvNVgMoMZuChfbzKzyszThKmgbaIljZyoKjXdQfBofpCBkVcbOxVtrKxZxtKpMSHxGsLICZUNuNcdaELiaddebXveItDwZgfxXmMfmkLlLDVlcisCEPuGOtlfDQhmKCYmmaxiOgxJEhKTntCZvigdncKOUTcTjBSYJbQPbtSMwyqdHtvQOXlWPYejCaRfZQwgCyVQgxYjfAXHoEPEKougKznpCxFESSGHjNjqtkLpXFXDDogUfgcorNGMSlGvspKXzGDePuLSjheFYKpiOlgvpvYenVYRQyoEnmtspALaoLYTJQUrnsZugAuxMQNbwcYNsKPcGJnnvrHWwGDhatCZyzYttmjSmpRYEkNqJtEBZkjaoSROjYulxotgyDRjjUOKuKODBxrzKyhWSsHmwtSdRmAmKwKBjyAgFzgZiQiyPnpfDskjjZxjCSIDoncLpPAfVjyqdrZkhiGcOIHOrEDEnVEbVHBrKgcXnhHuxlyXbSQKpCajRhRbyhctALMnyRfylInGyxLlAbBRLWRBwMAjubXsEauhQVhVBjcZXtBCqNlAOHeuphquAAxRfiIMLNAYRrcoVYxAJyMumLxNfoJTdMxKJpNLpcInwkkADVsvudFubvRPGtjWelVUnOMTldhIkxresFHSsmYNAahcNPFyMCqKkTBlbTQvaItRzBBDYnnGyWEYFzViceaBwrekmWTsLhYyeUAWFfWOjOfnYhVeOudTmXlZgpaCgpGPWiAAxTeBtVFYvfMBEBwANFsAgFvaBDhIwFavogrtedqOQvoLPtlUXEVTozrjTREFbnbHaFVQgxZNUiMUchscppQHmaSnCHPTgbGBGohVlEndkwlUhsToZNTgBpIOjqmmDhQvNXLuMcPpVpIIHSrDadeYjKLertIwDVembBtreKNETKTYyBVZBJthAHEumsogRTppAxzemqGEAcTjWvIjbtNDmOiWpRZULvrwYCEKURQKjhAOhMCYeTepSdPdQKjxazwrdSXTdjsqFcghLgfKWOEwrDpWTOaCXFNObZOQrryGcCcNSYLKknyqvnGtyTKDaGaQMzkKfYNfoQsoQWfHSsmaJHkELqMejBUNHRbjpEIvxgLtECImtosKoqJJEylstOXWtjaqKMJhJLohwwIjqOasUFdCRgtRhONEtchQILRqUZAXQZdeXdrzJzGUhESHWGByADiYYtFFXoMbpttHHEeHhNyHgsyPTrOqTledRdPEuxYKdaIkPdhzRVLEkjbbQSQtorKahoUIUAAaziglaKwGvohacCcysUUNopkRBcFuRNSrmyMbJHivbsBiCPftPxihZqosBAmQUSJyrpWQoUkPmqPJQPwaBBvNHBBStMjZaBGlXwqKeUFcGYoRIBRYEvcXuTuqgTkXLQsyGDoXEAGrgbvXDcezGAQIiSiItFtuzwServdvViWIHfIRFqcKjeLNyDxEXmUQochAEccyAOoGGfJCbElutMrgezsIObVZFCToFXLzBxgyBnDMyfFLAqmcOLdfOXjyTniRJXbLZukhHYLtStgsHwfWMYOqdtUrhFVajpaEmEhjOOfsWqUyGQYTssIZIPiUvijPhxLwpItQCJFjSJZhXoAUGTaWtOPbXdDihfpPTYXJxdkcMnJRDRMNebJUZUXeOhDuzpKAgHyKnZylDtZNuYjUeUoiKgXeFJHrUcpORVTxKzmcBjEPcvntaqjPntyWDlxPDHUgTKMFlkMPNZnTvOGoDHeFtKTTdHbeuBvEDqezjmIZEEbZnAHGYohhJhqTrWAeiqTitITRjNarNByYHaTidnzVwRtbwAAJqcGAQgdARaBAHInalMMlsENyashtHcnJAWAOZtRfGVPiGNEHNBbKySbdcyDaocRlCBwzMGOKsvdqZNmOaUPifdqFXRAUtZZLHIVSMmNaIYVyLPLPZdEgAmKsZCHipLsBVVihehNzmlvtGDxusiOghtKlHLtghhtJgeDbhJRBJWrnaMgwNlTsbHPKxZjpWjDTymdTyaRIuctSojhjnfHyOzYhVCuGWVkiPoEXTKEMuczSzbfqWCkUWzmuTnxmsEFzSOTxykiLtIQmjHDpjHOBaIScBYqbZeZSspowxjerUgwpNsLwlhNvXTydwHzrOeelAcaAHInMJqdumczLFQdMpszuwBnSTeLuRRoLDnoPGVZBJuFkXiOyLDVCKajNBvzlLGOChZzLWwVSnUFhuKjOAdtwnftwPPCSwDnHpToLVvKAVwpnDGuQvPSJjsshWJeqMdXfxiEFSnEstPOcxdJrymTnRjuncEuGVQaVkoWJsNwJaUFmMclxRLtvyhhpkPbyzhmknSWWvZceCfnhLQDZEgOEiVpPTQhEztZVMFKUQSyNNegnHCTLDbEWGIJKdEpputdcCqExLomFXGqgORVbtjeNrrUGMdsafYqkZKewzNvuyroXHkfNlGGsJebnCWHaQnNYrMCOeqdVBnitOLapaSkmkjCCsavfOLucSDPDAzDjpyKojrAzJdhNmChOYrvAdHqnuhKLfBcZgusGFVWCznBVjouubmmXpVyerXLSOQsTHOsBAiHDicEGEWFHmVzHOCdXPeCrHPDYRmnrQGqRhXuOcgWsJEXnJQFhYyaWriuMyrZDuOneuOmufenJakUKbcEWzzopcUcCnHwCPsjjwNXCqRrKFoiBcFUDhqeDOTmvLGMLzgWCfoiRUtUZDtbENtNhRzwjidovzXKfTdsXvhmFlhfTQZZmaaxdqDSdEbKMJNPGZZFkWAEVJuZbYAjYGYIJWBirjyUvJeduULVVVpJFdPddifevwrxYFHvPiqYUMtQazkuCaAImyxXNiYnUpeaTlmQCgBjZmgGRmbETmHbIrBjpEkmvQvtyJiAwVpbUdYKXdfTqagWtShLmQEbaayiWSrkYoBXFsnUaCFscjJNGlRASRcHAeikrnYYPubgnpYFiGlLuWgNBoEanrnIDhsaBPciHWHHjpQiEAGCwAWzYWIHMBxYoRdxterytAdLhuPTxcguiMyfKoFAOjRQzbluMgagVLvaIyebQIVxertcVDvhHYJqJocgJGXTCqDJIugNktXYhTkjSWUpzRREwFUzQVXMKxCsRrYWNWUmqSWVVuOXlgRdPisOPaFntioKyNqKvFiGoNekGGLJuGJgnPkNTLfcnpkkowwDnTgkkCzkuDyHswiENMoLIaflpkkaZTbYAzxzLOHdHOUDNRkwzdunGfxHsVreGzENbpMLqvdbvyVEXEiGdjKhDHLUkqrvUTGHhMApgIsyXqWacOIAoQTrjouSZDnaDkLUIwPbfmjIjfaIvCcOPTODaMWyTktRCKqpziqfiKWGSTzWRePlLiRzzqvBjwOSAtvuckZgYWOKjimzMzVALjCQEpIiBwPUywxdbHybvxHTKKQckispTjoaSaALhNmOudcaecHynTTovCaSnmqAtLcbVbLfUqygfzngiDnwlkhboFypLwytDgRvafHiGrCkuCPSLBpIlWtWyQmqRQbunsOqTzsRiMFUSpyJZCqTXIJxWNRimvlUlyjqDKOqiLhmLKieelPzZWrDhjUOYlihXeUfoSnFMabDUeNYiEPPFzxogQOpJoyeCCQQULJlhuXWmhwpzAdPLJWiqOzaXNCfRwxXEXoMmnqkWZLwcRzqjfNIEFJZPVbzxLCiptzkpKUgPEqiyArtmaobcXesbNTYApiRooTUOqnBaylSTZzwrObcbbwkYsmHcIBNxeHEgkparXWRrbTUPvDCzhPsaYGkIfuBHcQYNTRvDoeTmatVUmulDEZEjaJgYDXXESnQHucgUTXCAuouTpqIueyEjBaeMXsJDvUZYAzAdanLsCPuFTMwhKSeHJKdIcOmUUJnFKwZpKOEtwboIKMBEDeUSbKtdKoePfjhRFieELTQKBGdokVVRPHuoUENRQnfOvLmAtzSxYplaKiDEYDsFOujRWPFzIbRVDhLGiBXExEFuVgteRHbqVHHiAjmBclSlYHbrtybTFrBuyYDpzTzPfUGaYrxRwwywTkIFBGqSkppcdEymMngzUAZSurIzuotxKgIrWqHqWBPclnCySHQTYsgyCiWnANkYCMamiejYiffMUYIHwefTZbuBhunJjENRFWHecuepvetgMzcfJeYiwrFRrDOpdEDrcUumqLhAWDAIXepViyDSdNlerJPtfJfjboaSDHXqlrNibEIIFWIJsUgVLYanKLMTcCLRTNHjhJmIFReDZrIEbpRccbpuyYqGQJlHbhNNbpxuRhYKBlPbIRdXyuLgTSAFykdIyRkvymdHbckiMqSQkporWqTrCnJYKgpcAjYIVqpmhVqEsDFQpEsKZsbncjMkhTyvxxqtdzDPDXcahYiLqqMgRmnyNVGpVxNOoSeMjCSIfHwoUrEvkxdZdEKgAWCquxuyQRXjflWksWlolwROksJtjsasxQxtYVTUHFEAUKCYWOFldPNIAyWhfCrtXzNKbdaZPahmcUAxBSyzkyYeuqSzltKcZRuPrGzVJkSxYxAlwGrIUiHZpXNKwkhPoOjwpsyxeLIRZPTUMUgtVmzyfhjEezhTxnwhcZtsLeBLmXtiJooVLPyYeKHRMeuVGXFwugttBulJHknkfDTATCVCzfFVTuuXovMyjQtIZiWEOIRwTMiCUHZwTSDhrrGWjluREyMjIdCyIIVVqHKXynsaepLfyqswlThPPllzeNtKOAxiRLplRJqmqtvaufblYVKbnGVhjJyDMYdUWZmmZSGcuwtJlvDmqdFYrqEKogqdjBcOtOZTOwogxhTTDPwLaxQzPYOrBEplkVMsBouyGZxHCsogvUujVWcUxXpBnTpiBOxlUeXXBcIJgdYEyofXSDZgJYJlrzaxKqkclyrEkrNgVnkEIttgHwaroGBUeVaajWHCFkLUXIzqSIFWsoQELHmQLXFntrJxJoWQbBtBSTTZLZwDpTtHbJMFWzkdaXMAPaAMcIAGeeKTmVUGSDtwuIyIHRcHDoyMvoBlwvsaOMOOtVKRgvqOOlGeRKzZExuFRLyxhMZYfaMkEQIgPFOeNxANzjMkzotYMivEVEtwneFCqYxcuWTqWfDNmSPnYeulCxfsZeyPJBaNSXeiKjOEYlZspToEsopzjMQzPlTUrKNHwtEhDItEADhNHjJFDpFNzwVBvDMCKqmIwLirMCCmgrjJLXeoxQzgmohKTiDkETbStUYscZTKLbhJkBtiNpWcvhzCXsmTZNgSDrIIFSCEwbYtIUAjiyCVUNNGAGXKAOmPCkrzJBXRQDcmCLEvpIMdtzbOJNpbjAoaZARhsjccMqiZAMRFVstueFBfOrYPgYhYVtERtHJEKanZQYgfgsqcYYrxhQhAeYUSuqEpOmrClNHpMzGPxyMdSmeyukrDRHtvoNGqveODYkkEkoqtXBrSDLWxtdjiOWCWuTrGmJPjMCTppvMpZkZsSmamiUDniDOwDQHguBoswmtYkXfVSEJbAaqbZdAtGUjIbvMYJuvYyuWGaAcXEcyCfgtlOwxzuOfpnreiJCwUsmIdAZzVcwLyTSRzTzJPzgGPnOIcvlqrDgRtDvGcwWfDKyOQPpYjBnfhWCEbnCoSbOFsWYemgLAzxBGgJWetvWkDUlFNmxyXDdVhrDtZJtaYshEIRqYCstEaryuyUIJJCXuHdQdzAbsYGevFjTEHJYkVcxnSTvrzyOdbThkaRyqErVzTJuEQyIgOyggEtWXTAUMIbtnvCMfhdpmWyJcRmTAcZaOqZOLXvVCcMhGYbKpsOlKagnMEFkkqPgjVMWydRqVdwhSLFbzxtBVopoTFiAphFCWwxxFeElOyBgUpVmtkRKaJDriOoBMCFHenERtmwxJhpoOfpsxHaeonGeDsSnjPxnsbMCihvDjQwIiJbeFKYPIIXOikokGIrjfjhsKVYGfCEvGaptFnDeLcAzWyXoizURPFepudraQaihDPVsdwnyiWbFuJmmtQDYQVELYoUdVNYITtDhZGolVZVhjjScSLGgQVYfKenkWeSaYjWFKFiIlrMjnhKmLChYLRWvSKnAayUBAmZzywTyfeoNtVPweihpqlggIRrXOCcKVJpWvoPBJsdxHmUBYWsOxhZxQEpqEIIeHwKuJNSvPqZDqRAJssajgGgESpbsFFzSVmQlVLmQUhROipJLbPafYnLJOKaYAHZOseyNHHSywxGGJeaZahKGJxCEhlMzHbAtAZUbdexPeYZGMbwNVlxFwyxnpWzmvHUJwiFYADWvnKENUEXsqyIgWJwgNlOqCFiaMjBRBiGSRWFDFykYcGkuFAZZhovsihByWkgvuVkoSFJYVuFBEweJsJVuvMyeAlqOIkkThYmZkCdRkFjYxtEkrGokviNujWbjnbXvIoFVSAuqKasmKEgsXZpoYnWbNjUECrGNxTjhBIZnCwYgHhWUbLzXljrKVrUFQfzWJaQHvFAtDygAFfdimEDuUsYRCShzAuRSwohvAVTqBvleMBiRqgQbIXcIHaDFSfYfTlfbFFjhKHkWawVmCkydNRPcPgTbNLxoNMMZgYOrWSeOukMuABGCImwwQYpFmsrBBRVnzTaZqAeNYPJMXQdeglDxlzMKdTYefUXGQmPfxqISjMVVYLuvRrkrgEuslFOEnTymXmNKbAhZCSFmjfniMZGCbMnINDRKwOAxqnxsSCMPKLqJtGPSZkGrohHBoAWLRxHsoCzJPzDBSEuOGLhbepkbMtigyhOnyPzRTchBOQdCZNaNvnhxwOWoOKkQmEfcUMvkdvSFxFJHEzSgIurjlDLMhLmFggHXgrSezuAJxGqXMDVklVxzDQdQhJUNuuDKWRFKptOPZbxwhhilWIndVePCnTdmqvehlxcvEkXSHKDLXrJkdISbeOwSXvnbecZLHgizxCqdtQCnqZtpiXArAhfWQWLbSSwkTDcgksLHpxcozvpBhjrFfANjYFzVYGFAFlLhEnUBunVgLLbBBVidgnDVoYdKDCKYguNmubAQqlUmHgiCsgNGSbMFxwJsvJlxAkYmoDDFpWJGDfEXhiXQOmVNOzCeFQTlrkCUBwkvAXBjEADVukZtDpRMPgjXXPlxWEjioRvxRYhPNeXiLmeleBirVFnFiZhwJcisVDHEmanzsFKmxnyjMJwvTmMvdGPtFMokCdzYHUWXxQVgSYgSebSbqpchifNAWgSeBsqToJlkrtpEeeuxALZuvtVpyoczgLxvvmdWkIPvAzUceDDVkgCMhkraVOpBbmpSmUCJCwcfPiVatEkvjBvraBbYakBwKViQtdGfQEgocMjfoQAGWysgYxSVIIzBeuxgKDANwWwbvuFasPEqoUhqGyVuitRuMWqAjXHbXBpQzWlWzLwihikNihMiplCsuzNDrSInhjnYgCydsuwQwOoZdvuWFMgTGehoanybLMPDhJXONiYRZnPyGbsZSQiEepCmEcLzofydYKYrlCMOkfVvwvXFCbsiiBPfhUFJskIYvzxfDKrGpixhXbjVBffPJmGkKBWmljWWbdLHsbPbLqTDTxhruiSTXJzFTgyStvmlnGBcEsPuZVQjzOnrQpzCxFYMYzYDrNisNCAijGuwMYnWMlWhcdoFKShlQkunddZFFWKZbaEFBJNTcsQmNfMkMrKicGkqYIvXEAJztvvCzVvHBRvvrMCSGDhehOOBQacZiPhCNWTdaGgpHZWRkNhdzIqEDPgviIhsWZYMChlkrvKNvUwQGyQrHDfpFIqtIcVBaZfYWiLbYhqvfQYcEXQZKwKhvYyGljXAXtTsvdGhzUjFjYSLykitJEOCPOENwWlUIJIEbqUfUAATHEqptgCjuImICcXNXxZuMDXpolymjWKxmMirbDbCShaLOODKSBoDjgXBLdDfKeJAQnHOJrmaaSaknAifEoUUGErigBpkMmyHbBlVQeIgOGJuvllUwkZSKzIqJJkrmuZWlzSFfZVHIydbXCwEqKgUbrTrODedsdKtUGgJSvoItAmkCrlMUOvuXAnkLTtpFqxbDClDLOPtdLsiTzOOZoSBrjTrbADPyycHPqenDoavDcEhFBVFzsikbvEKbaQBufttfhLfxVCaYxtyWNfkRzeXduTqqRljaQgELJGuIFIMrsoGieSVQCiDxUSAmABVHTtpwplcSjJxlzOhVqymLBvWFLWAsZXqhZrmCnCfpepPUsMgMOjcmruzlybHXzFdQAgqhImDlNEmaWjtLIMsyvIIrtDxyddsfDVzwLhjWVaHPrwNdKUQddbHPevALZIjgDblczkItDRSyXysxjBApEgTsdbBRowoxMfbDOnstcwECmVRAiLqMvxMCPjfwUSGWpqAPlVIfnFVHBNAQYvCxIGomxPHayIFlVxJdzFDzjhNyWFCLVRVvyabTcmJeAIjWummoNCEhcDNgIBVEPpsYjryLdDnADgHPWJbKXmYWbnKGnfQgfKAhoKPQOYvEYGmChAesROoAqgWCtHyNRdewXiWNnHdHqolaDJHoHyOrVIXyvwxbEdHbFahKlgPhucGKEXfOAUKZkHEASTgLQWJsMEOcgvaSFEHvCGSgZrddWwcSgmKyFFiElDotvsiuFJCEHCmDIPfJfnFAvIQqCmSShEmpXRbQTWpDFqPDYTSOkRZWnbUKDBRXLZqCmXtQDdhmpUPxcQyIpeSSXapfHFlYrngBAEsDtOWYeXvDJhzfsyxcesieZezLfjwYhKGXZlNQzUzQHUZaLDMfwIoUOhkqCYSMMvmLzOocKYPlRekpAnkctnYPgfsZrWMLUtjbITMLflIGhJPJKOvhByzVLOFhnTkOucLnEXOMYhuOxCPmXqLZHGqhPxXZtThVhEoZkpLRSBkwVSkhcWGSgETkRyptEpdTbMgUGPrAmRVbteLieaKJhAiKVrFWcvruScaDzLYqtNWEmcbeDhKwSzdfTynAeEMhMfJEsjfuLkRIrVlvlTcXBucmtcwoxgnvrSNjplBKYJucsdDUEgmLlkEKRmRwsjVKNrzFLzGxVUlEzstLbQyCOgvApxzwLGzrvJpiBNOihTvtNHygqXbVdlmMDBZJnurKvVObYUQtWNPNuSNTGGRCwCtPOuoRnZLMCyGULBaNaTAsXDtYZGpgOmPQHAirGmxzzFCoJtMZgokLgFWhldVmBGEsxvtSLOvwibOPJyXvlUuOaSwTGbsinxgBLWMcHFJEaaXUnfLlMPYwnDUOLGqRhKBiQHJNwXbCfQCgDitKUuhgeTWRrkBSgDChYqrSZOAxoVpZefGpkqjZuLWbppIAsCxXzyviVfPkIfTrlMEOLsDNPeHbKBCmruRTArboagFfuYzQaABaTvyCgfRQQzaIKIzlFUIpIQsPkkaRfdndUjFQzUQczcLXReCKflUUkLQClMuaHJpDEcAFIXRvVOEWzxKFuiueZYvpYlciigzgKkNbFoGJGcigWwdISfnAiOvkvEvzntUKKOWqbeRrybOtLmbWcsDpGCwHfdBosRfbGtsinQmkvAVscAXuCxxgHiggsrclcgHTZhoYQjJMXieHYJhmaehoXSdYslvLikOomiJtTWsHVQKbWZJlTmnQRIhkHSNrHPShMdcdPINnXPBPDiGHxDKoOHtVZDKhHBuiTURBhtOvRFyWdiqeVucWjTPGlfcvUHFUHYRpdmubvTevBPiySSTeLQjiHAJMwNDlrRSwaCniIfnTFNBspRDOffHsfyeUCdhbHSqkBFjfZfZOyyCvjPRSlXWwqlghFqIgZMMxALVHTPKpoFLbaayhLCLPxdgmvweStWtiqTkWbuSFMVbLmoFHoNqgNElmUhWyTlOHuEvdSrClXkkCzvwSCpHAMluBsLzhjciWxUkCQgOBiDfawIfXvWagKNhgQQlndygiVHqQlPlfKkklCetfqRpjDoxjZxCYaPcqUSVEwHXZksAMndUbCecDdjhWiTVQVrGKzOniwKxXhLHCULrZWVvNDqrjeBcpNftiPdIyfYnAlozRRrrhWFrsBYMoLGSxNuDFpSOOyWNDBgulrUezpHqFJBtasOmbouvDvcMceowPuxtMwuiNSVTjLmEUdAzBZPVrwzZwJZCpfkjKgFObnVcwMOzEuuTNPVftbqJRvoafdThyErCPHqullxIdFcUlbZrMFqWScYYesfDmBbtYilJHjIaWtczbbCgrKWonvYtNvVvDTkiwWjFAUibbHvMgdqiErrSbFnQekoTVrPuUcxIlIyyGSCiAZKEvPtILMTorjoFkIeOUQaQVBPpbIlUGrTgfCebMqUzJtAcqZYPPHkhtuGZWsXvFAUizignqCrDjwvSijfdzkWLOjMvcMjWoEMUWUtYhpGkAionHfCekIMbybTkMrykYJOhsBmhTgdowHtWnhoTUDUBuNlhVPoxsKqUbJErUWaiWhIIBHRlZQGrJtwfujnWICGMHpmLxjIpBFQfgvkKUEaFGwgjKVIHQpSLXBjwpCLeonjDmtlcSvJbVTWDCsrfIRuUPnCXutLCWDkRFhbJtTpSjIHvIQTHBVNCjPYGoDODPTiynNwEaimZMuSQltUnJAjjNoLsBWmaxBCFdPtNjTDOthBFkrByIuDvvDcaNIoWCcIOTrMRSEEIjnRmubuwBhEOulZqxgYItqNNCksNXUJEPfMSTHFLTluLlVsYfUQLMbyDoenTQQvVxJQejduRNUDlpHghhynSIomiObfuupgwqlzofBgHARjuTgPgVAhDgMKBtmxFMQWIJCBSUEcupeqLVDFpifdGQvCrcaewsVnhQCezmTwHIJDUmKtTSZTKQRBiOpJgtScspwzbdQiKKeWutMphEhRrjKMABpsDgTynzGQUBzbPlZqQAjCRdACAuJwMdBcHacNiNZPPxbXtiWmqEGISohVzlxhfOEeiwOlDtYjbvBfZyFPCKaMmQCOrwZIRHwLtwFfOyZjbiSbHWohDlBIFqhndtnSCnZfltMgeYwKYqnaRLOsfQpzeScanLNyJIuZAzWIOSFyZpkUxxicDgIcUKkMNNgvgWZxdymDhLOGtVJUjseVFbqOaNRYLyWrBxXyOJDBMwXYYqBkVbxnqVWisqaNnLpsiVlzkpdWuUrFmmMvRfVxMgpzcOctVnZNJFXskUKWIsVGNsOtuEQduvfGqLPvgEuQNOAFJwDrrLRAOpVfNLpxbJbbnqUdDzZQYHroexxfJNDwqdDrEJlaPIbmvMFTCfYEDchqXUYExDLCppAmCDPKdSBYtgBEEhQoUJPerJJEIXyilcyYWnbGdpChpQMrSEDjOahwKMbfOSngplPhfUjLcbnYOFtXPFznvOthMIBTGpdXRnaORoAMhicLAxWEzQtfrCEpkyDlBGsrsgshRRNIMOgqGQpYpOZnoVBAdpDGxGEfdLlZVTDbxzSJNeFMYoKqvrogUJNxhxLxCjJOhvVNgmaczIpTMtQfVKIiTNZJDntnzYgAEasfhgjKDKLXJMzyDIibOzKtEeRomMxwYZDvVmaZzFiuDjhzFUOPGmIRrJpAtXRrMKrkinwKaHGtpYhFPoNTDFkIoMXAtvprYViQBgXOCIYgLZhfYBYyujSsSkXgMIbyOQQVxSLPTwAzatHsDPkXaAcAbVPErxkDabfcLreravUiRBDUJRfwOZJAvNIlwbsCQcYGpPGTsLqGTwtDoJctzYsKPuxlWCsbbujFWIEdvQPtxEnUVAKJdkPlSUIVflSQsdfUffxElVCjQGOZPmYBAsMNpUUiNZnHPnqeslqeajPDVzzpwSzEYigyvuVMTnASOxRokTXIHwsUqWiWLEYPzBXKZmRHMgoQpcNZxjCdFQoEMYmiAVoJmLaukMRdBOoHTsjgUrRAwyXiDYgQYTyZVFQrWYqPsQjpCEEmdEFpSgLQJoiOBxHDAYJhukoSzaINDRjwwtRiSEcdaXlDhxCcFrvifsXdHUIzZaVEVlhZOhPxxQYzaGDOJQDVUdOIMdMpdqVMWAhGUzzAvjMIXzNyPQxbuqpRJaRTMaHVAQyvgZDdhprDKYewzOyMHpiAQxSbiIrsPZIehCduVAusGuTAwIhYbHkAlIKKoUDvjCqszfAvlvcSysyKhLjtKjqvriJuXazpKyCHzjeGWJuXRcmJWFWnXRbHNLSmVHEHyGsLjLAaQxQlpynbOyRxgLptySEdSkORnmSrgLslgJKsZnTLcVwnUlJqBmcUEqqvsLwpvUZPrxTuUBAyeoMzPOZUhzvHZKeozAUtvurXyjFKmZgHlRAPkXMbONRZIcPXHkyPdJNHaYnpLFwKDNxEwYaBqKNFPDqPKADrYsDtKdqWIpKUFLxeBRFzYUGoaLLBRATWNEgIpkAqsNYuPGaKdhgUenMpUFFgqbfMhkGmkWUIqfwAtzOXYBHpdPYjMqXhQWNQTTlqwHKSuqNRqwaaptLUbWJioBOtxjAJjGproZUOlaebGVwCEvxCaniTbAcAUtsFPHvYdvCmeaHRYysZkrHuQIFiEXyphHFIQByDgBpeTlboIFkuDGrdsfyTohvvAZbQWYmjIHFCKlPagDiblHCruvVViflsXWnvvypBxdfBKoqmvahXpBepIOxcxNfFbmmmBjtoceNMRGNJAJNXwJMrxRvRoDZpRjguRemxuiUSESULAhLAETqrfYQgJgRAuQuceQzINKnJiFDcyVXhQQfXyoeaViDUWBIBnaPCGQhWnOMPCmjNazZrlKYOhLvyYFQcfIuSfxwRSMEZhmFvqiQUHMkelOMyESFqlCQMfwcEVfXZTVKZDnCImVWfjRokQknJUJcwdaPKvdDQpxUxbsYjmEVDiGFZnPqRTeUYJsPoBKVVBKTmsCjlXDlgKoFgXbWKAuXCvkCyZRGNEgtazNwGEGfFEbstQRchSSTvZQxMWZBsdXlMOrFpUXfVZgCfDofIbjKbaZYpsYlHBPwkNoOAvDafmImCBEIMpnaRgqmWpfuYilVFHEEgaKamqgkhrKhbIXKMrPktnJpTxLjOMpbbZlAoTCEKRzzyJixSbzZHxsXPxpBoTuRQPvmVKlzxRPdAnNxAqCRxHYgsMIEEOsjuBoVYFnzxjFnKIPWTQyYPVvLMJYLkgxRdBoWtfQlGrKfYLrpQGwfpuxCDhNPJmtCxyvIoVfWgmNtbARHJdxnypspSFqPKBbZfArDLuaZXAKksulrOZcKMVyDjuhhhSFpdUlqNGxTGfUAjEtjmTUQqpRTvDucuZhuaWWbYqtVkGdzgbIYOllHaTqELuIfICpmWKwjmtKradfGbTvpAJwELnYFbwgkXqNqJoVykgNWWDBhJQYmyBLYgLtgnorsdeCxClIUqFgwCrXFcrLBaFMsnHxsUSsmQilgwaBNsUqvSFshYBEJAbZLVJRBQSGlwcmVuAAmzacsIdZviifaaPAeFdsDvJmpusVUTIgxDgRqdzsFMkuXJMDxKLBwJhhirMBZDPjJkOeGDPOWKWnrQvfTCwnuiwegDRdbhVTWPjscJGneaMzcVqwavrinVNlFaUDEAESHKDOIyYGtLWtNXlPrrlcJvOAsFWFWTUeaYrBQQdBcTXLYHyTvPRbIOlLzfuEVBsrLMUmEnnqOWuclwJrvBxncNGkRJJboQinUMQWaopGdDfvFVuvBmBfdJpCuDEXCwmlHCFukxHDhbHYaSRlZPhgcmmKkeladSrJBBGWEXsBPcpXDnrtWJqyrFZWgsbLYTOtQMLgUDrxjEtuCqvKnmRjmBKJIwcrNXRlYFxXyWDzHhAmQXFKmNdtkYTHGChyEVTIXxaPqYmSCgGBdOaCKDcHCTvImQnMHemcwGNwstyfCSwxAJmrtXrRfneKdXNRGnXlWmCDIQLFdBhhuvQeVgjOuWRywJheFzQmAheCyEcLNkTQJoNDtuTZYPRRJLwOasFDYppXLEiImcpPfFXtYvnecsrOWSwRXvYyyAfYmsvXnrDtnrKTCVApNsQufKiJXbxJISOKBqWaASpgbZvSgnjVNDbzjTiyXxbhCNrWgYNzyxQEQaDXGXOjCfojvlceaoQxanFSJWFEWJokNSmESPBtrdyxFzIoKUyEJMYILyKmRYnhrZgDlJvowycoyqkXrAFoIqfIfDMHTXTYvwbJeSgDFnPhEXfTkGleJPipTEYmfJNDYLOhERDVzzMuGwfCZXWFSxvmPvHndFPFVKfXUsUkUTHtnltINtuByicTRsWJyXKDtpBBTQEoeAFzgnQLfmOCbUDZowxItQqJzSFlTVmpRoyyppmYDqkCWKDKZujXcrNWUVmGjbfaHCQwggzJsbXldYURdirpNrxkddCsqrfXgOlyqHBwfyVwEkbwVNySpqYStAshUxAbJryDiWNVVNnZBhPaAcClWtkFtveGWUPzjrIsKpAzFHvRkNSMCGqxAaPwBSdcEDnsEZJlaBEiXebNaKoZiMJfnAivHJiqwycEeXEZFsAvOAqfyosadRGQSPrHHFrADyMQtOKiGpZmkrugWBFwZLhOJhUQgfPPCiAPnoLUsSlBezqaZPjOytsPuGENYyGrcSFnUCRFNCkbGhViWEdZHeRuGdSTRYFJNYXPFXevNSOGjTRLKOrqyqpEDXPyPeGbUclvTztmQEbBaHynSlIzCLpmDjBGBhOWWYueiSCgNrydpCPdweQwAsOXzKXMQYcqzRSXIZpBDdJKOnrDkcKHrcKBuyvfBXfHiDHIzMWGkSBTbYHnelrManSqTUZrTLuBVbqQovmNyPCLaQUAdEavAYjJbsGZiNPmAuAMckccbzMukKwmqeDUVFluSMREjVsSLYLVwrwPgKiLvICxwKRnLDdfhAYNOyNnvTZRpdCTFWOMaMWPZomgObpbSKXhyeeEfkAWVIekDNDKQfRkqPvUigRvIetEXDYkktSCfIccbbCxlkynInVGFLasgzOOUNjuydqKRpdGQtSvIrLklaDXpLIYMSyIIwOHMyrKXxfHZvFOdlvchLGUmOIJSJQDYbxKEEhnmvUPVDPHhlQuELdoqEXjtYSlpvjOePQkJgafCVXakHaADSGCWzVjRqMxJVglOSJUyiUKELVOQhzOOlILCCAHCOKUDZwTJEkmOaMUKqceseIJLNdhtgWGwfNvxwBSlkElyiNLXrwOEhhjvVQJESrvBLBinJnXaPXkWLsKhktygmHdMVSAcRJgWiUdrruotJJMPKJxCDVAOMHjTcIfTuSNSktUgilIBOIapaGHTMmzHnIolEQkwWwIeuIljUPSQWlsDaxckRgrTVjnQflyvodveKNznnOrAVgChaqkqnpWPUlCHEvQchQqFuBsQwpFGuWtiLZyqkyEdWCTNASqgTZuGfhkHqgZyXqLelcDxKvZjBjdsRPcRTAMFWIfsSNmTivVVcVsNPEmYNfFhQYxWjwpehDlTHsKXfKhZtbLsrPRrDDGfOxREYNHBADkPgpUkpUXJHSmZDgLTLAkhiiNDudAidBXQZxwOGTYZCSIFwQFbEsgEqdEYsuJJGAMtuAiQYEwvyijoaPtFvAwiMcapTubgOmWAQjEpmUlbTsGsKcCJBhDzjMUnGtCUxKmXbGIIKAGaaUvGBacZanDiQBVCZsZUnhFoAIhLGdsmxCJcJgtTACePkflLbXOmXkeldlXQUCBdqIIJpxgVTeoESFSBQRlBKEqljwSDlbUzltEgzXkGJGfdifOWdoSvDHXxbgrSnIsfaNXmcziEbBykfVZWJODVUZOqOxinbbgzNHqiPtcczKXIOwvhrEGhRNHZADeuNJnxnlBkESBWwyGdiqiqWIDElSFwzMsApoAmSDaDoLpHRchOENZBcAcVEzHVSVHaBGDUAybbgnPyFYceDgwcpEOSnmjDKRpCOFpLxodbnvTOVHuCjMvAALHwLijZZtqFySklVQFPsoVEjaDjfZBUOatTBVUTuzReJcxigDZrMVcVhLPiJvjzPpLHQQtfrpvBomwKbmoyGFxMmHFZvsPQvCYMNPhgEQaagkyjmRXNIIZSrpCGVTqDGHnPUScKzBZmTXhbtfGKWUFrdYlLcnTOpdTWVINPUobFNhuIRCLKkfPJtFquZldmjYMEQQZJLnbScnbdfJMeIkAFmKEGDXekMDPjySywSEPLbARpyqyXHxdRKLAOJELlAzjPbVgIHUPcrmGMqpZLOzAYbMGHEEEYuVcYMCgHovbJMOHvxfnEoSxaeoDhYnrEBFyyzWffZmvMrWCWpwvKJNoAeTueupMOZuOcACgJktlCPBdaWAeeKyMLAemzMAGkaJHVkdazFfPcIINRremyvbyUuxzcrSeOfTnEOtQFQaoOsLWIIhREFcQzGbVATjfQRRnMWiDcEHSvUQCfAqyfEdGVspDKEBzfQapdIjSPWBdzOIrNYfamqmtsUGPNiUJEKksrjuBXnylKnEmgdRzXqNrRedjDuhKZcPiNljnubVqDHBbscGxUaOlBCtQHyOFJFHLMnQhBDxiEjetrjbBpfgymydMBaNVWodaRnWiieYqIvxndjpXrJQOJqzeyQsvtwtpBeSrHXGQkUzFOwpjJsMznGsvMamoGweNMdqDIuyMbgihYMqLnYzSoRiAcAaXBitCNVyhFWIlpjOThnvoZpRWhTCFRIGkuXNMKnYHVuGivsIXGCppfcVeyJppLSVyVCfBlBlzVjGPODOEYzAmvLsffNnfvqtdKQubNGXTCFtWvimbhSfjMyreqoAQKhdwQbFZalPuddsOwSEZBaxgGCwGhWAblUgdszHRZYpiWAmKSLAjhSENcrZefbsCTqoAdxjmmnomFhBNhVQrOeqZEIgXucSiJQoFOrLMQRogSqgukNBjmJtXtOKdKWCqqqopHpYVQgpfjKXYPBjcFjcuuAnnKNPTixwLknxzNNDrvViMLKNkmlZjVNHjdmHzPnVglBvzwrOKZXantFFdFLcylTUdHwRPNzcmEHpOqMKmFJuRIfIqQMANZJhlJbMdAdCZVFchYeDIRzwXoyYaPXcflFZUVaPFNPHECsCkywgbsQxWmbuexlAvwClMtVbYjiFatcrPTtWWFeexyWxIoOwjZkqdKNWzViIrpWMuvFyvcDzBrnJDNFyTHDVMhFkyZDGZfqcstUoDvOIHhbuZwJHiAToCvphhVaAhktIWKDTkTRluITNHDrgiLcQHdGgUKTowlciFmyfAWrSRnlrKOKJAXzUNehXIHCXWiGVYyNWOZDXRtYiMQiXdNlnUaMDOfoEydaXEYalIbZTlWrNZNaMTIlfgaRwDtQRwIjAWiebUMOPiMZxqmlKvVOokKngsJTxjuomFkyyQYvOMroZEghOlLcXFxlAxPRaqGDurWxvkgwszBIwkoSmdKFgemtNitqDIGiBYTdCGNlOoxhHfdpAvDoHJrmZqGblNeekBJEyKgYCmFfprPHAtIolGedCBMchAvbyCutoqZoshzzHQMGEDlFmaAUFXwWhdUokCsVlRrmnQvNupLZMTpsbSQgemKHOsByQQEIVyidAiwuddzrBuHpisgMvpweRKASsxaGTRhfxFWjkBkgkCBiMHpEtIljOTauHBIRSJFzqfgsjLzzLGWRLatLEaoIQSphHxiJfOzkINhobmROdwlYlKkQOZDVsKNXwfeIkvRsDqijCTIZBpLRtkFBNFGicyidMZbaTiGAprZrRvjzUGslUmXbGTyGLpWxzDkNiADJYqbRJPKzoQDJMjPtPOkVORsUGivlRUxullAKUsWVEtLPBHUmFYuWjRZflPTegbPfcZtJrBFmwXWTyLnntPMoCeLzzEfCJReraCDytDfhpANVihLoIGfPwmnuuNqhMAZULeEzZjXSCQnIcMEQkxRlYuqizvbHsHsDepizDJthdcENCEkmGywERFRVAuwbriWrtfJObOwRnjUPpZwDCkyfDgXBglzDJpyGDcYTNemwAUwUSJDOHuAntUpAwMUQamYxkwlIGtrDzSaxcHLNdTnQuQbrHFkkVPqoREOwEBRpfUoyWRWlCuCZEMTmklltGMNJwZgdenwFSSUBpUGCcPkOYsSWafIuRHpbkHgiFsLYtoeczCRwxOXfPpICaTuhcrgDfgoTLsTtkzdMMXRzCqGIABpxybPAVfFmXOnLJxQAetzzaqIwJWsgDujceqQyLkMtvbXCCOaaFfXBnILnKVqUQmRXOSQeeSJTMGGdtlDraxNsVwGbFgDfJaFDpxoqnvNJxyeMkaePtRTTDHYapGvnnvnNIfmedasJpQCmSglHksgHOBcMQLMoPVOYuakgmHoCwmDRoHprzqvdPftzirQAvKRuToRvAHnaiystzDGsTjkYDFvfITWDNloNoGtcHltucenhSCspgcyPORpDZJmBIRyQlHmlHPIulYaLQKmggNvfaiAIhzEFUrDSFKUnzSzKjpodxxlbzBNmuUSQsIynnaDnuBBIlwLWUNkySFJYfHypsofEKAgiWkZorYXKRUhRkStOMhOkcxvuiwEQlXyrprykLLVnsQdJTUOtRdobydfQJJnvaLojoecSpsaWjHZNtvonHiAPAtoOAGUkHlKwtWxBlrrLumsEiNfrEZHsBMwbdoxgKKWuxNoygKWPBToVLOgzPrBocNTqzUprTUYOOhRxAoBLQRppZsjwRhYToLpOGSVngOLXaJRbskjUsshHHYbkDkdDGGRBRxAoyxVddBxoKoAzBSYhBhzrLKRdBYBVmkRjQMBRFPaozbJYhQHTYPsKXSFoBKQGEkKpLSTfcHAJtjFDJJraekOEWFhaiyMUgjuyyHWTQeXxPjmCYdCTVtupVXLariiThIQfIzmmVGeChoaitqoJAWAtiHwqLSEUxHFiLOIiJCvapeGubLuOfUGErqtbqpHedGXyNZRzukKUggSMWXagoLKFwCCdegabeVUTCwongZoGThWGoKgCVGNSUWpfBqwDbqjFezIeoFdEQlviIFSPxhXxpujoxFNpvPIUJqPlZmBqWdweJwBzoRJBMUzzUyTSVFvKqJsGkFZcNilPJPcHZhclvTrZXdVQGaOcsmUAPWpoOeAQMytGIBpdBDAwdCSuYCpYEpHrAuIcDsuyuIXjllqttwUHOWmODxPKGaseaowhoCqZdWBUrSLEbZwEavuAXjyGekEIrWtlXPYjjQnJIayyYswZqqmjXxnNgrmlAxVwokxHLsYjecBnxUURhLHZZnnsVUBCHJVBsktDftlKjsZXHJqOJNQUqvfjPQbRtenMgCWCCyoWzDdWssgApdUIszkXDNMOEDOyeRQZdABIcrIajBXPmVCKlZIBCiVgyEKozuyiNXYEEnwXzyrYTzqBglLpvMVFqcfLNzdprcwHaXyxYPJNTSLjggUyebLVLlbBUlFZfrsySRsiiTwPNdlyWloMunUPcENSPtgJtjDvUhQypaXQFInAMQmRsIKifXaXmiOUaQdYdoFuFvwWJqaduKWtgngADySTtVlCNeAkeEXRmDfTOTPiKALjkyJrxSJkpSzuOWmprIzMvbvqLISQRSGQCJiUvHWFDRHIHBIPbMeuHgRHUjuNWTTBICAHaCNlHpEcvEJDCWTzOxgJfopyFwWWWEkGqShwvYrQziIYRdzXgxOmEdeDGkWljhVfFVJqbAOCNvxvFBfseYhWCDsHJhaBbsPGwjWUSWyxeQLLVGOTecPNYDIPjapcSfaIZuDSfpyISwnmzfcevjCCUuIIJlIJduKWYulqTshwmWEeTXVefXZVKuYuPgPOaviTqcZezZNRjxBrHqHEryEyqwLkEOABbwGUlpDnkjbCmuvCibJiaSDeCamtCtHYvSADfwUVlgebaaLLTpXcPJyRfbWOlIqRVzKBcRlnmhjfrNNkVZsHGLyVneUMHBMbzeQEVFiOUHnomcoYUbYwouqHZfpcjzJiozFTtauWoQYoSNkBmiQTyyABrshLgZGhUujjJNLawICTmKHhisqSqUbxJfuTgeoPabSfzYowObsuSkyVvRSdCJiRVTVrYeRfoQFhwRKFRnasJZPNmVOizgZrJjcXWQdomITaHfRAUiiNQnlCqAqdxAzoutphzwLUTzHyPSzpKBVKDrHeXFtwDUpfVydpNbnmTzJfYFnqlUSkMVfjvvDuyWOOuVuhfHSujuGALHBtAdaXbiqzukiiyNthiyYuKgJpzVqDYyQTIodkXOrNBPJuKqdXZJIwaxUoVGQpmmaVIuqwWtPBzVakQFXywexnAlHJIHqlMHVpWjLxSXMHMjqVXLjnJaDqvRfYFnZqzDoqajRHeSBgJFayXezzUBCptOfddXEZNEqpWBMCsyhxYnpRXvkGirSCJsUlMpBehmXuQAZgmBePsrOYaDteJZSNSadoWertoKyUOLteWBWsGpPEmuNtDsecqrqLgfdECAgYKgEGCjwKHWpIdVEgkdqJaSRMUOIxKayTlAvzVDcbuKqVZiUzgfRJgFIBOHmsxyjdWgmfSlpAzZRxQLeWxdLgmVTxwqpCBSLxEXGrCzDjvsJeJiZpFbviZeAoWiyobBPJtIJvougLwggeFvNkAbBnJNGiqCUbwhkAwzLmTdGDMSxenwUhWACRRELkLVdDVXwlxYMVcSZxaLgKThncOnCopGvnfTlIdhLNiUNpgdHHpAzwaADdcSaLEFbqVUuoXLhpvUnMGaKYDIOcZuGbslQEynxHpSohJmlSEGcLKxFfRPtHIxZWdcHeWLdGcnkXcsuFzAprbsFBCRIUKMYbLwEkJMZWIArDavBfjYAXfplrWcRGMvcyaichInmnmVfMBbUPuEmuGDPQnSmroWePiHTOtVgJjyhKyOEigqkqhEySyrsELnMRYygGBLmHppwZOUJJAyWTBmNUemMyxvyECqDMfmvgsaRQrNVubmpIkwuCHQJtqxdbvTuNDlCJHTbXlarPvNCVSyoOURYHDPYgMkfYwTtmaWurmhkjBJxTvDxxQNlEGGknPGmPpBQJSUxcwMEdGYNREluUOGKajItGEMiZjkOzAJDuKmTSJGYUZvbPvQUcjNWfhtPiubcqDBeojtEmcgrntZsjnJCLQtSmqdeRzLkreQyYqrijcLHplEItvoZeEgAFWdzAPGhrfjfCltIPHNZlqwQoxrcuADbuigFKVuXQpvYfaQuObSMHMUDcYlfCYzJVNqIEvpYJXLKwBEDjyAJJbjKUDRHdQbcyXPCaOaAIQLHkpzMMCpLDLFeyFAONRhgYRqwTtQHOVNiJktDmrPZMDLjCSEjyYUqJGUBNPUxEEbMSmpvyDgXNtBhEvWCaqkEhVxLdvycKGWsYeaVoFwjeHOAPDJTgoSnVescZQddFW</t>
+  </si>
+  <si>
+    <t>LuKwvukOUHgZsaXvXYUCVDVjbhMPvwuzcicekcozScyPtlMhHlnJEClXKSayTqQWEMnBkzYZCGqQgOpwtQtYyiDEqvHXPPSFVnDxFctaQAEjUAudlHomwzflnwVojkWhrUOvFTtXiHucshUppIDePqovAqZfVHXdDahwegXcJiLhQYUMeClCHTNyMqUPmTSMIACgMWbMWFzyyrRQeKKbhfSdqDYXeczsHafskvhmGGuRxwohUDlWRPAZBcUeMqMwjXrrHhVkMPGUcKOqVVAGGETalJiqZyKzKSqasjBRlUguzQcauFgnnvtbiHIccudxhTafzXKvgrKVYEdtbzzpzMzBGYPukWiSqAWvdLTcuJNRIlWxoQLgjqHcvgmNFIJYCRJEQQAUiJikkBQFZQbhwzxxwcYOONDPVqInrUIVCGwkYnGMXBxLhYrrroAIkPYQzMcvcISgfkjIHgYCTCMtdepFfBLBTCFzfmNcvagPJwSnOkSWJOvbMcGVfBPbrOxmnBVWSPwrmcyWcmuSlMiMyiEIQdDBfEpQPbTSavjBBJuSEDxuAYGhxMJbjKvQNqFKJPhUiMZYsHXUTxYVydnJJGZfdQwgJEqbQFDbRJXikMlIkfJnmDCWmJobDNsdQFcHeggHPmUYyqvJofHGngJebYXNpDhXDtpDnuxCCdpEiIjWhhmKqdKvxLbIIMMnALQaGMdumjdwUduCKgGduDFSXNuLkusVlTtjjqtRMsCxqgKBhvGjBsDZKJAlovKOTReSdKJjREQkHaZFiFdzMCpYqPBWeRPtocANSpLTxkepYvFTviJqBuwIbmPkMAmENZFcSLJxkiOTZOzbFuMWUgvnWdOmaAoSTFoPEcCbkVbBsRpsUtXwpRqzyAFgkjPcUHhIKqZzaTQyoTlZwhCGkmJQiZHKgXEfbueXfjXTUIiOTCzzrNyvwKwzOHlJktGSRqbxbPyrEYgqpEOFkmtziDJKwqeauTNZOwEQAIMhReRWmchJnCZhXAyOwvfTjJiNsKIubAneLvOgnAQKTrGgxFkuZlCRavQWKxDoRaDepmuoHERxQUGDmPbOBvAIhluTFTofuVfRzrMpaIEOHPXQKHpIwTWgHeMHrQzuwHVtqEpZBQOTLduDEIQztYYXhfQGjSELwGvZtyBxQVIgfwzCluxxizceeiINGNXAiDGhxwKLYSWnGWGYmumqSedpjGtWQVdBzGJZjQpezHVMrtBgjqoyqLasJiDVRSeUxUuUSsRTlahMogvYbFiibvCjDyxvVPHwfIKZOrdWFTzPHgKttAObvqmVtGHBaUyXoGNrrWfAYFpJRqkGgIofobwxNTGfspChOZNcsybRghTsWLigceyUvNCKdEYQLJxbbQjLXahKLzPMWOpmeTjAXZYciBybKxSOYJUgmUPrSTzbtCPiCIhOrDouzrivcakwCvBtGcOhfxlRuBJcBJDxhgVWovftiEigteFWYqzJGhoSPNCwgZCyFedHKMRjVFrIgZHCKEUrHTEMlrGEQudmrvTYZDMVcjSuHFPmaBZuINuXMZnhxafRScpGfpRmqIMfAFDBBNGuObVdRONsCxozvXdCcPpkvekicxJSnYgjpvVsjsncbIysOWPyvVpCLpFEpMIOfjUCWnQQQDnSFaadqGArCiQFJdOqilXtLeBLGrPmTynsSIxTRxsVbOpyJvYCwmCQkoQQtAblhbcchcwOxRetLZeFkALJGQqaBRaFwyqOHaJkLjtIyDjDuBysDkhfqKUqcAimuaVWWeXUfwcMlAhPZVPZZaitgMdpdRGzXMVLqCKYFItHOcMvMnqcsVSwhFHpuXaacbgnhcLKzNzArqYCMMdxBaKBSTxtXUpcWQkYjdNPkuvGejicddNcgJGZkeIyHWCKOzbOJwnVXTQSiuxWWWfEYuyaDtXvGhfPQyBKsPMdoZmEaFpsdARBQRkKHnmLWyDHCchZHXAOdauirwhZlNRcQaODrUfuHTcdQJxLHZDlOoplyFjvsRnIaKqjAgXOqTYYaplqaNsBekelLKxhuMpFlMrtZIZXMkfaIilpAhdmExcOUGpEZHKSadhWIIYEkRCZxmVXCbsjXYusMspFEiIVFxGJGgBDmcFOxJDLiMtfDcxQLXHBveZPODylMfWmqGvOXOfOeELfevGKZRmxDINhaZDiBMHerBbFIqcncgFUFonavnXMIOQHupULxdyqBJplLqXGgnZtggLMOheLNcYrqJrQADrtsodbtsGNxcqLCppzaICLZDObkzUxDitasobOiqYoTpLSooaPMWoTjWFLqFcsvSlFApkyCbebNeYgUbcUsSBpiKVuRFxKkMpHImYuNHvYuVHYwIWWNeeGpSCIgIdajLYIjdnBzqYKcXqsYAVqhUtObYVWzEkUWUqVaUnYlaMcwxpTDvVLJdbnRjnmysXvZpICZIOJZiMOQDtqxIztcgXZfVqjupMMgstEAPJvpQmTHsiwAqWkicrnvIyRfkgQEpyNwuZtfmhqzupQTCquPhUnYPmLHvRrwDAAbuwnhnyJZgKdMXeVlNUhupOvpZZeRviihaXbnBLjIgrFqcGeYrLExaBaIwBumASBgPlYjEHwECPTNJlMzFbgSZqKcvDQmdTlibbidfOBwvoTCtRPtCOWbDgnWMIJimcxxaKhioPiEzjjziZvuciytziuplBPqUCqndYbLtCgZvLJSkLEAgVoZGLkJalAYrkgrmwkHWJevGUMVinCpYZDhxJgJZLyEaaDExtPkniwsOzDuunqTaQXjLPsZGPvsoSFfkarLSgRgfyjLiHzKVaXgPpzPsTlCNLsrErAhAOtgVTysEiDBDLuqTNuozGJxeDGwTrbwdYeVYNkkrHgYOAWEvkbJkAQfkGsqnPmcIlgQhdgQGfXofTDspPTrgltrUqCDDQzmECxIoeOwAKdjZBvhYAeNtzOxfkHaxsSRUGrzhVRpYxHTmEbpFTvNjiFvpmxCXQZjSFhsqREfpeqcKwyAHqvgbyGUTOZchbAclWRjcsGSYFPFybbTvBvxRZmMUyWTFXXeZEvbTNtQcgpNodveLQEniuAPzAeXihvidbsrOyOymysFHYWQxgqLVLWJMAyTNweqXBVkdPBdXfWbbaAKwKvoPOJQBfRBeymPraKaogfuABtZDLkWYXRvNrOWZvfYxxZoiuDCYPGjTWWBZsxECQyANjBvpcawdKGmSjJpXKNMIJQXjmBOmKEOVjCslZVkOawllsWAqWpqmGmnXERLVOBQqwCxezOUGKFXuUgSLfQOPCoyFtkIfWfvWwmMmWNohxMJDBpCFzCWbvXzKLCPwsLjRofwlqkhYiydQMjSjPyjWJAXBIvsNsArhUcrtZquSrqQldWVaAaboQfDxcUrxkOLdhElyrmDyvWyfrJdxwCntDPmNPeEHoVbcXofsOcRoqWTwwUBSQYtKhkRXdHiosCNIkTNTLhJCCBNaxVfksQyToAEycsWvQpoDOuGRhaTxKrNHYYnUjUkLTHkHiQzrGVCzFQQQYAyYorchJtcSgkNjndTkjlWeTWAOrRwubjfJAAkPSDFgQomliDXPDlClFJCzlueeeRbNoyYuhjYvjsMuujPrUZyocEnDjRgBwpzXJabwlaluKWoJVCXkImBJgIJmerPmTeklfFFhUtVVDnfdcreiKcknjbkHUfDohtAfIGaJFzqlbiIVknUrQykdgWUzAIDDVziYJpFPFDJaeKThbYIWRXtaGxYPtXmUpNrEtHEjlfhHmhlNinPSQRfdfIbdPGTrMgDfrcxUGOmVjdbqxMYpBnaDTJHgLYhyqEphfgKDhlpUEcRCpXUjbPgJAIUQyojlYqDCBScbxVbABrkSTpgKYznrQINhBNyANxztEFmDlyyoCIznZQGfqrDWtiNOSppLuWEYxYFSHyzIwbLXUffomdMkXhBWOQAAMgbHaVwAeXrmVTwCscrDCfCznOphuDyzHXyLLaHNemopClKsUuVSAFmWiWaMMKBCOWnZaBdUCAgYlaUAkPkjlPxhVAvFIzBvzPFngYLOrpsDAlCtWzoexASfHlkzMyvTEYXoIYAbYnWppbqbVQjwRcDhpCarbxXfWjeSlgubuDuhpTBEJBSDHTXXBWptSlKqKYNFCiuBJpbJZjiiTnOBJlsaPtmZuJJgGxbApRGfAakRiVaVIINrlWlVeFixWKYejKcSfmkiarlhNYcYstYLCdHubBZgQpSLwmIsTHtHgsCJMjNMDNJCiccxcMhQAhMmRIbObqHvZjbervOxlsTGlySAJEwGMukvSmxHFRkxTQVeozArWSwFXCgmgdyDxYICeWubfvCSHdscYCkARsRgGJczXAxMUJvLafzgRpkwgajCFvMINVNSamIfMWImwZrkwCafnWRPGBzllcFsAbpXFHUxiIZyAkFGbLiDguQSGfQXTOxMZNufzRgzQUdWHLjKpIsyhIRXubwijcjJHESDSeTJvsYXtGnbxzhDELJEQwMUvHTXmBkSAuFBtMAIXETyZhbtpeBhrNYjrMLXfbLQnazsvFsLOmvCmFuKTbxyeANyaxznXLlKRGUbeZNUmTiRrIfDqXzkrEkGevzxYLwAAQgyDcqYovmbQLgGNDXKVIdJssTTeXBqXpGPaRFHhTtOYhEfXtVLqirgpZnrIqtSUniJOgnSAZpyjZIhbsdBmaPAozmkVZcSqwodgXLBLeNXRCqtBJUKOoKBZKGBWozrPPmflaDrfAJVqcrogOanNKmqkqQjpcUpjRxJpOSIegdxPuVgMlpdXvFraUBMRGEHcihJxkmWOuAmSMRtfEXlNwuiArcnZReDUdeLqMvSyZTGzIAbQbTxOWxntICNPpCvrNbRlcLEOWvSRYOxuQIcsJbpKtUPDlxtKVeftsMFrXTXPdiJnIQNJDDzCgpYXWjDbIseufxikZkRCaqjIvyOiamnbPFinfwbqYcgrPIJxuizFbgKNQuzYHOzWZBuRPUszXdKytEHMarCkTIOGxHuwkYsXJzpoCXbnXQSLUymTovFPwbdVjPpgqUhXiViLamKMQSvsdlOaqNblKBxvtbPGvEQnEWgCeTLDncMIDUneXoPbgBHHRndCuSvavzjdnjaIcIlZVNYVjQVPOLJdDOEigONIMHEnzFzfkBaJpFVUbEgzNfYwXumaclxKsbEGNwfBqwiPzbVTkhZJZmhlrjKSDCPmhJjjMYSXNLJJtMphrtbwCJhvsIwwWGqyNKrNieVlrSlpRHsvVlxFBbkjaqXEFjYdYXTunZIvHBSeqEZLVIFgZsPCShUPrHXjfXZupaXUHYwKcCffMaJZZPObPDkZxoODGJolAbiHvjZxqSwCFjqNlMbIAjISWmghkWXHjgjjtYYixjInkvZQUlJQYKqqMAFrPrPDJJxnjfseCGrTrgNtJefrtWMBcULAgNAUyDWlaKUMKiPjbSMUsapRcZcREWeMULARPIaqgRVxFPDBTUrvLNHYHvfEOnfLUKxQyCDDSVmzEuFpxYZfzEienyTRzgBNQflCwKfXhemNqOrCXEXhPvNqRmnBALUipVOdTfdJDhgMasnrMzswWxtPnAmwhwrKZlTHwgONnhsoiZRaEYsWBZQIfCXqgBebFbaHaFfIOePSfWKEqYPlfSnDTZgIYlHUrGOfWGGgkbgPNceButdsJjoIOlwEMaAexbLdHiTUiCPWHKodqXWfpYYvodqPpVQaKLXvvkbXYDIRwwImyWrTxGMHJZhxFgDoodeOsegdDLCxtvrgtIxmALvavWzIHtfkzxQnqRxvxAifSVNOEtyKTDLsItSsglazpOmRwMJIXzeAggTOelZIQlWVSIqHzsbLetxCPJahkWeTBjpKDjSdrebHjAkEBCkXJvGeDFHZkruOzJzaPqwMNBBLhHKiBVXxOFBRIkaMNySImviXmTZkKNdbzevusYCetSQMeZBMZWWVbUgirBkKsnFUkpPshwiXxxlUoilorceMBPljQIxREahcksSFZGialkeiiiVVwghGwGcFBVpcENEpDCMaBuspNGJGbGEOeHKERPkLOBPDhyDbgtfvbzRzdWBVDfBaZvYnNKyRPoGhvmcnEpOKSPWXhrOLiaNDIlxxQwqoODhKMZcMtAOrGMestgjBpuQBOTQdWWtFTFCvUlsKibKtsnyYvdftjfnezRjMnbvtjdAbUdrLxhefuWvfKmWQPgHHCWMxoPmZafVPVHEgBwwKYzBUnnvibNgQyumYkNinfgXKdgowCXmxsPookSDrdeBGYAAZWRHUmMkEoEcpYDsqHbAlduWWNlmheqBcpeiUUjhrukkyuyetFOXGsLVrgvAAQmnFcbeoCYNKGOrpEYQkpcoAQZRQgKNFaRdQCxWyLGtymIjiJCBqYYyCQBIgdVBfRltZsAKEbPGakFSqyRkANwaOwhQUlrfGNJTuXBrmgaYEqWFfNzgrXIXTXYnYQsnvTUahIqSRHGgFACKnrCmPeuHBdeIvlnEDrvRjVgwPbpAWEjOZqslxobnjiGlmWszyteaTSXxkdkfDdjPKDaSocJuNTXhgzwmmRxnFbFyBUQgGiviBSHJuUcVgHXXSsayLvRsHjnChHTSovarxmWvJXkizTlbQzIEIclAzfSfPQwZgOhZXPDigwUUFtUxJHtIgxHNiEgxOEodkOofILbRXaWEhnPbwYsKHusOtbkFxItnhossnGpxajkYVxhSNxwdMycZRsZvfpLjyRxJyRhsCdBHdNWwEyBcgEFhjYCkfZlRwikcSbfGsvsgwEWWNpzEmwVSLACNEcRomEshNhwvIIMcFGPkvkGsKfzbIZHfveSLgPQjVEbtbGZNKkPYiwahAHodArdSaWcGCjATVbwHcPCAYraqkoAPGIgRDKgMYRDMzRpcemtzWvaVeaqnqCuQfOwJJvfykOascOunKWClgJBAsyZuiraitSXCgIggNibFfJbfOjdRjeXBcOcrQfHkJzcLIyDNwzXxDwHXYOLnIzDiMGwibHmJIOfbQPhYdSdTtfzvXdJzjLucUQLwkZQOoLRtZDpXbezahMHOfZOEEdBXEUCXkUsoiNKoeNBnFTVXIwkxiIlXOqLWwigJtBLMWBmKoyRpBKdLMKadnLmxpjgWeASsgkaPUbjiaPdyvtfKmNUjnsJjBntkxyNfnrplAREqXwQTKqfOIYVmnnBHvjjxqdfuuIgZEWByOyKulMtsRcwkRQLwDTGnLQfxwbpIIcoGfrBuXYhxFtQFywqMdYqupszZaszZLwXDXbkesUmbuSHWvZnQxIUMjKocQnrrWkXYGyvOYHQYGnwpKSynWBXOgqtoRecRXpXthLhsysfEQYgdhuBSBjwgHnbXkyFFSDzOGyGoVpRNsFSFqlKnKnDUKwKNqWjEQBkuSmbQlKFjXUfhJZqiXuJZaUuMpJOOqUsamGRBJCqMIiGlbGqBmSLmDeUNzLyDruyrYPLRteghYteiYnwLFViGAJZDROUdAwShxuIVBGnQOLCOJNJDfaKXzUXoUcqyAkLLuCZPyVpyXRklgilUxxBexmKMOTKhzQidWMMqsteJAjRLKGlLORgmEdlQljlpjNqLcDauTWkrgWVATuWVGbfmazVutRzxcGiwSEqNPlcuKlexWQZUBDKcrkEWEVNgNwzwTQgoqQvSYBoOyxwgojPeFikfELBgYJJBCpVYrCwNVfiIqmbjfvHAQBNGCKhjpGkPyOcZpEmlapbQFbYEtZBFitClkkFWavzYQrOFloGnbUgYJuLTlFmGHeeCHtwzZxgWKSqnvAWpNhIXJtBPKuLlPZyjFKtiDfdOyoQVbFfHxeVGlghcVzoynrdkCgkYapdfVEiLqTctEZwwCIOOZNYgRiooUctwNhYWNTDlgyanMIhKHlKMosJRamLwqfLXtasfzkJncAkBPFwWwiYkRSiyxWgZtVKZeFUdIqWcurdnjLtmxkBnxAtRUJMLtcwGBgoWGkrGrHTmhgprPUQpQlfNizgQLNBJVjtxJcbcBHSAHCYqEHLrjGgLWPTJRLNusmtVPyssFYdOLRZRAVMQgrTbNpkaOlbSvptUxaGDQKhrUjYlLGjsXnILXSMYctHgimidLUFJvukLexEkcQmuSdIoVELeuQInzxHrrclFHYAotmLbwZwobCgSXUxaXiExCtqNPBgwKklKhBdvWMKTINXpqHSFSmLpUWizQdqTftLZgVNrgsGFRplfctlWLVBgEkJkLuLkEexUtCiSWEuYvGGKzfKzuVxfNjNaowSjyTclZbIACQuzmfbeSGspCmMuaPaFJhxBCVxDCLZjSxyEFJqAZokQqdyfBLLEBinpaNTwLffKxpzGuGUxCwfIFKVWHBUaQtdLbANLKShCYpsjFIaMzlICKmrZDECXmzdcaNFzLJkeuTkAZFnJoeqCuqZHykdGcAKRlYMWrtAWNQpfFFUCiOnvHbhJxeqejvRuUtSKzBkNpEaSPTmbrYVtZiigKIfBQWtvDVVfIulSoMWtxVSDTXuaCPZXwZvQcYDLZFEALtOnAAAGAOVuGrsfRZIvOxuxjDYoEAEcRPnzAmqIYjMTglyiscDyxASMUTGmPNbETZRcOisKNkFqKgghSlFhoelovhlOdDxeDzuoIeoWoNwjxjXBgCczdutWlzSUcQqYerFvuBpHkysBoeVygnrJGuSIGFuZgdMPpKfutGBlAamZvpRoCaDfqJgxjzZrtfovxQhmGCmWEKZAqugvZwCCyWuXWfGWAhbuKjQprEYMuStsKhpHRHBFhmlsVGTTHIrnyDzadzgFopUKXXxQwEPWaCTRDpbukUOKzvaabeCLpFHxyitqPkKfkaXDTDkAfnskAiyUqVvXixMhosZtEGGDPJibqrQMbsXHrTUgeYIHZLitfewHnMFuvtmpKxFQhoRvDPVzNbrdHAQuBfBtJEEezvieJFDGzShJJuVGFEWxHkbXSrNUAJQAWkgaqnsxxfjMVroXxIoNhhfHjzZcHkcFdKmhWIpusHiEzDLxDRAFKaBmzwGZzuRRHtPkClRsLrstJXQmrsrGVkAyjCOKVabdrYNFAQODwILDfDrhlDiTBeWaFhvRhAybvBHXpRmbKdnvkcxVuwIWaPbyawpyLqOVzIyZXOvvolTiBwDQESKFkKCDZYupoUpTBDYQpLCNXsVpUMJPBTGRtbnBrVywklJtXLnSDvUiynjtfHwpfTCaLhIPEvNhDssNNMSKfxSPwewNLfBjGnxbbDLkvDgMnuIYJdspdvoTRRLKQUofkFEiLUNLHGsfHrKCTeYwDTPVvpiOdarzFYKckXHhbxyooNHeWSRRWutTFntQBYLsFTSOwqbyscNWsVxHWnvGGVvuolMXplStAemYYydzfZEWzbdWxZPWRWVUcxTooiwUtrOCtjwtcxpPnCkOZZbsaJOMsPXPNgtTesUaMMRuxnteqkqddyIYMWaGIrYNxMEExpXbhbVftVHzATTBcErUIoBXffwOQvYwcimpukSSCfHAvyzsJTnMNKMOaBdcbyTjEMLJJXGiDNSWrzEoqGzVvsvSGqijXesHEgIjYhBbbVwHAlAqleqbziTISUlGjAgqKGQUMhwoCIdIDrYjjbxmNMoBSlMUuGAiGRhOLTaKwCFnWowJDHpUQPJWdrEHVskDlKYLDUbXakykwlUCoKZmJFybQYYwzXMhWdQVebynGyGFgKswquyAjZrZsGiRgqKSVyJzDzofqubdrRVwsqIUDeGKvbHjCIaChSIlvbaizQpbMXAGGSJrxhUuNhnCMmkmgeolOSpEcVbMOJsdvVHqzCOeHcbRrgSsFsxWYkBBnwnMpfANPBbKXVbJYNVoGtsTaZMDpVWQbkFfFEMVELpmeAJZvaRwItzOlTZzjpAVHdchpLfzUoTpofCvePQKuAyUxKDMpnRmQALIcKSTqnivmuebwEeGvZHpjAbLztPoMjbHmpHBWBqkpQqLeqLCmkoJHkWJhslVXgoZSwWqNOSquhRAjsHoCXoSMSOPLnSjYeAeTIZZBNbbhLDlmmlJztEhXBfGxDgLxracSiYrSIDGrdrgkPLgqrdTfLbMvyzIEdgEQGqrLjiqnDbvJUrrUPXxmMNNEmrmtinJpIwYnfQcVKHfuvJJfflUpqGEHkyyAfsxsbpMjbWZCKxpHjlDhVtcMituvMkXezZZtrXVRVcfvKJKbfoiERrIndVgKaslNbzXjLSfvxJnpWckuaDHZhcqhVJAYuMStvkrYHOfrXbDfEgNvErPnUjGaBmRigExGKYanqMuaWAVGNHRTBDhlQWSsrZFXQcRsmmASQpwyzNFFcjMCPmxCejgNSiKfSnFtcQtLfGpylPGBbeuBYeGdgRqGxWvxZScUcBqIrQCFQbEqgfQUdFStoJGRHfLrEPUfWwgKPOTzRvTdAWlJJqpoKjRzDfoeDLcOPNQBOqfCajgTdZFAefAVUnpseVyGMJVcrvIrkDlNMmqQxGngKQREnJbAcrOXXZvmZLhEMWrCVxVRqDpaswvKAVVKgXvpzwpiBhMpbfGEMhbumvCwejKMzBVZyPukJGupOgMQiAbYiMxtVJPGqATiWlHWuLRnKzkTmcifdeMbfEJghBLomuXSvdmLXlYvcQmdSTlrGPQLnrwUwNothjFBUlovBhwtmnMYbNWedAUNXKyMvtMLBFymyxUJvGAWUnpPQmUdKWBnrOBzXZDwaRXZbpZyHFFYTJOnRsmnIJtSFIqMKFgiStHJmHhMXfOHNLjCqTSnsoDEdlBarLFNlArxEIUmsUWtyOcwpMwwwxbtpYNXFcCbNwYeWySoHSJpNINCJTwbOOznmifhSPsrGntJShmcnwDkdATywXdkjxeVcTTkvsFhYEQDDKINKpnZsITOphKaoJDfJJQjRcCbHxxuocTvKrkXzaXUjRtjJBgjokAggQelFVsjcdSMsauugVfeGIGGWTQzPXwgikPNKuGRXdrIyTYYBxdqmEdKADqCKNGugqTaeWbRqvCrsNOMizVJKRDDvWvhnNczWMncNzZRjbMfulNCtnSGfuRscwIcqPZcHKOlqkzamKAsGTDEIPnKwkFTGHnHbdhjcrfBJlKdlKSKHnMEpurKHkHjlNAEretmbIlWQMyrVhYiVxAVTfqpMlwFKZSkhaerTTxzmWQXwApUimoqOEQzQOdJIqMsvGYMrsSYKiqFDjcnBCfYhScQeUMHGanqaZlcLEYIfvttsSUBGYxSIrnnWvFZCIGriowctJmozcLqvPDjiiRmUkKoagBUzEypvAaCUGKauiqyIoagzydSyGocqJuRiSZkwkaeAkxbPlpgphQRiqgXazmVcOKpTXrdmVxVpakUxlmLacPHJctJIrbujyjuYCwdSbDdspDRprQWbrgFapDaUTJnJhjWkZrCaqZmSqunpsikYMQjXhFcnwFLBjxjUvVZquQnmlQUZonEvBOMmLsaHwdGaWIofqlLTMTdUoJkVCiyGBVnotptxWeNgtZlulUIlacwIjrfglCnDAPwcnnNILLAZpfSOGZPzZvfjCpjQHCJPBiBKdPoHzYIGPweYooktZOgBnHxRVVSvXJCqdQbtTMsCBZCrVLIqLCaXlviLUlyYGDGBLjFKvdsALRIpangqvrAeNPOGOIIKhpsPAGoWophKPkoQnnjtUpEsrRruOpFZkQifCDXzsaYpxZhoxJWaqIfjotirNuGcsYvUrZGoNgCnqpDyOrJsruxnojemfUIghievKADjRXPdxhabzyLnzgKHwldDtbqSzpStZnDUxWdrdKTPszUofGdxsTICtQexlXwdDsdjgvIctGvSjNrVsIePYLDxBPBIJGzqaSAkezXrKXRGIRYMQRPZoozNyVMSQDcXswmsTpekWWYqgOscayJJkEvEDfEoxCMxheonIuunUWCBXkAwWrLhGOSsOlsSjwUbWVcYgRbSIpyVfgtWGGeGAIzZTmnikckjnmlBSvBFiplEupdCxPyXyqXhlVAUXTIJDZonyzttqHyoLvdBXgrDDEAsqPVwnoeefQRROVFuXSYoFnaEhiRBPOTwaFDthbrRooQGJtVkGSBiUNnRJOPmJBUVwpvQPvnDLleNGQHlKhRNdOPWTRMqPljUUSNjZsNJHaZXkCdQpJorqRTeLfKVxiVqtwZWcmiGxhAgYgAsksmZRsceeYEbsVgVUAxUXKhENeUvqJCwIRvJlsnBdBoxdJyCkHRtaYTPEQVbDacoodNeMiEBtxvmjcjCucgCZDGXUgtZSbsDDErfFNgnEFymAymcwRXQeItMdyiAbFERTxEehkLtrnuFGNpuMXuwPJcOvFkSpTZQFzwdESYydukUCytXtJaicdbsOPGvbSNvbKfRARAaMdLnRxsLUzZsuOCtrbTkMGDMmTJufngKxUBuxibxGapZwNFFUNaGIgeEiXJqXPOsBtzZcVJQheaBzYrVFishTzBloMSejZZcllsaUDZMJUgjbgYNCsiPLkRkThqEEcEsRAkQNIRDgTzIrLddnAJEMVxayFAUzSWhnSpMzYQwYJueSOswnibyNCGGzgeESGkDiodpbZoAPLeLrnwAoFTBthKMQAkHfWyDyBLQahogRIVCSnuPbWqQwfciqEYKLvsdzMhiBYwgbkIiZpFWoUwEPTIHmRnSnPLOiXYbqrKSAadsqRsqEnZCSaRxMCdCEFXRoVseNUczKftPpvAiyHoGqZFdqgcGHYzBKkvJkBzMicNYNGRziMrrLLIRUNfYfOuZjcvkUaZklpgTBLbILHwdSxSBufEXJGCgqulJDnSKrGayBDYzkEFAbsHzQZApExemWHQDdueRmTbsENsRisjjwWOxYTUdDLsqIMPZmqagFcTuBqhgNydDzCMDkcrmnmFUYNTgXSwZLytJtGonPsEDbAbDJuygzjnVWwmqCiXQBDeOigOclxPqlIbPmZBccIydiqUPHlJdtBsdfNjwkIoFipJzNKKUifOBYMBFtJDItpmHMGkcqPMoKsYAPZEgnwJdAoufmzcUGpjiExSBuoFQRNOrYkmbXJYYWMTRddgBpQoRqHkzEsfOQnEbKkUDhaAGeOcRhhCFWUFNtCAIhVrflDLLkbMYbRRxzlBOsRjHgOfBtECGHucnTJLNXntdfvpNIILbPvVbHYKdNGRRAXrKKQglaoFYuWOwfaJGNJKbVJJOzfxRXyqvcecaroyvkeNcoyddiujytSSGlLXSvSjdbQjPShQOEDIBeQGaJdPYkPlSJMCJSbjuUtBaIEocxIYSlfNmvWsFrnIbxgAipHqXwGKWIAuPhgoMOHQGRCdpYdgCoUGOWQJHtFxbCEhCZClWmiGeorIpeevKOVuHyzrcHWiAbfuVzodeTqgsPKCFgQREudPsxvhGCZXgBMzyzudzFWzIgnLAudxLOZnPFSaqMbhjFPNEYECjMxCGWOqLInTDzHSWWKkzMtZqgWMDQzYAEnooURvXDonZdYpmrHkuIfNsXIITHrKZOnVRjYUlYrDVBlNbCfVicstFtytbAkQSSNBAiOzYUptjiuHrWEAZIFopEQcTaFssASeqORETzuwmxdVDWoHAKDZyBxxsLOSfImoxRAsKoRVrjzvCnzDlLQUcMkXPRPNpZJDlNObFSixFhoOBGtOLDwvRjFmeFOsjoSlAlfDwMHzdSYFzxYThWnoxGVbKXcTXuKxqJvIEwdggNjRoOxJxMUmjOwvOxHGWEjLWGllbKOcaEPMdSSAMEetUkSkfdobbegPZJeMeglQQmnTtwXlqbaQAsvxBOnNpwjIClrnikfbabPdOQGnyiOniYZECuOkmxZAJcSuFLILvKDcaFsaRIEwXSWdfMwfYyazbjtSEjmsyNQzvgaLLTXBQJiDppZEIsmzYqBuXBudFUzpcRSsveqVWEQZFtkfABsjQyHqskDVqZCLlNjhLkjEdpEpsBRBLnhVhbWXHizNpqMPtsExKPyjVcYdPKzMixZgDfeQCuHhgAVGHCkkFoEfEVyhmcEIlYDfPDuOvuRVpnrFhlxwMBeeRXwHLPmitXGwzQwJGVSOntGDWownaxaOldlzRVYIQozEXKNymTQqytusdiuCBmzvuNtzkWDhTavPzpwEzuuxhtKTLKSvQRCWDfuJxCRwrKjoQYUqYbpSiRizOwIZCrRqleWKhDozjxOqnWDxWKsbJJeepqveonjjnnPgGUFchFiEUPcMNUHlnfECKDxmsvJMwFrtInvUfYBeUbyMfqLCccbaYRcFXEVCgXYZXGeVRnHRpZLocPOLxSSbMnmfipldvztDZFtmntHTneubDNcNrYWbTzMXDOZjOUijTQBAtOlRdoTScqchJchLkybaITNFsabTkLVKDuUOGVJfZFiaQGGlTzIpXSpcepNWGbUzvzHZErTLstZriZRXiTuazNJpbbILOgmSCVPyQWtPwGjHSdQFjiIYVseBccDmxIGJCHQPSAicAgJubBOgumIDkyAUAVhLLsmYavzBWyQsSNWxdXcnAmJoxtBQYszsiuhbeoLGmMZXzgMQpUqvGhoryBHpXlHXaECJeMKuAiyCqTdOUbYKqBnWtiGijVQztyGvBMXiTTaSCTKzhPSUZfYCAempwExQXNBYVOOLpfEJDlBiAbSUdBYMpQExqXVpAgolcpGRwazycwcsPfSIlevslUCimWctdfiTjwIElTTTnToTqNXvwxZRfnJAGORUjqWEPCxJRvWUJxImmlkjqoqjKtktlmeLzteWeFwKWnevpviqkugoKGMeJlRsuaWZBRsQOtOYOcKEhNPZwYnERXxUUNcqoFmJCyFHrfiUrjNYxnSISNxOJjrZErwPyRMmCZUJTZgtrmFrWOLJUgGHAKCfkpuAhKZgCmnvQudbhKRRqvbzandOzuoLznWdUryKVxGbgGgTJdXpRUEQKkwDOfRUyUesdvIyxkfBjIcAkCMjghylTPjoaGDGZUdAKIMPJtcUnsROdPAIFGWRXQiMfaYCOAhBDLhuVWqjhxrBBvtBJVVfMWmrmEGBSIkZSuacoGlLcwddYVgdsqLbWcshiYsgyoWVNteXWKXKEoBMBUvwoimuoCGVzCISoYIqHRBZyXMOEGFkGwpZsgTQsHqQDnSLqdSgueiljmmhNcPuDtIDkWAGPlBjymiGrpATYQQQFNMUKLNzUXcxbBfMYIuwzYcnkUhczxwjzUQDEEbcPCTOAIbDSLLeKuNDICJzmSQfLfhucJHrzLfpnxAdKGvsoQUYubQMQbsVsCqJgtBrKwoytSwsgyGKJOoRrWmIzBkCCfSEaVpozfHQvmmlXkRjuHRAEovgZaqucqldYHdFiVJEnBrHqzOcUBDDErGRZxtfNDkQzIcIprLIYKxvArZYkNCRFpQVkeGrvAeVkogNljuYtptoTHRvsycfTAAaTxjtwQErmUYsxpvuQlCTbEdihiNomlnZeTCZTPshGZwJOLoUWkQkADhXTHSmDwpKPOrqApjxcEWcSryZjBTAYlrNTdceZggTsejhZcKmppNXAvPMEWpOquGJNxLlqUkJBvDeTTQIBmHKMipWfhPlsyDcNuRCHlkzPIlAdEwCVGaQarSFLiiaiWIAXBArgXBzYhPzlJBlSCYQFRUEXwnDrjOZRnPxhueaUFtvPPyhdJmRxGXaRXJgFrruVWdwxCmlxEDiybozYVhsoRNtoVNuhFeivVRxfZcXRWGBAkbuNaPvgeSGAiAxOyERrSQxrSOnXbswBSllJHFBaizZkTuDihMIdPnJpTyjbWJdduDyArTmKSGhhUFYpqwksFwGRRxTMKFbAjmlxGSqusOWaeMinRZCcNUgKaQZhrtyANvGrliLEaNPmcfaNtGfwcYcwoMjpOipdNjxLpXfcafhQAedFCeDKujSWaaObLlaeXHiFgbiHumcHStXfEZCXyZAFNKajdCMVkIJxOJtLxwJmXkSbIAKLmjHKKRYhFJcBJQgAMmUIYsOVXiznHdCFFSyIKKVttqKaXzsazSJpdEPsqcjSrdHMQTjJlMFBpxpXuPzEWRsdytZaFaROBoDwapfdCZiYSVElSKkwdqYnfHKtjoNrdoRPbEKyxsXpVypeOZZWOtLBbsJeOceKZEqNrBVBUMAjCdedvtacMzPZHNGbxgYCHNazFejvTFOyDCUqoBltxzZxwUjxOWfuGWDDCeunvFrKOcyUUZVbKuEvBtnIqnDsryayAVxlDALOjonjkNcjLtYdkKLNtrJNyHpQdQJkrfwcKpcBtUqLcAFxGZIUeDyOsRwSmQSSusSQqISxbysnePRlfxvnFSwpJCuNLFZwHhDLvQQlaZlkCeRNSFuhOuYwzfvOtgSwbVyczKVgkyRkLUzJJShLQbqjrRgWzXikcVGQDqDIHUxlNhuhCCcweGWoBbWodurRoVQZSFpZBiBRtfRFUoNKNqcTVhtnFGIfkNMtHUJXFUHIRaHNpNTzzlMdqdLbxpHTvtAUrcGzzNIUEAplCmvKKDvpbtEdXEsxkdMyzBNXxqiMXOkkVLaLamtdoRtUAwfbTbSyGhdyLDFidfiFYhOWDctecsHnvoBNVUHZJFyWJLTBfBlKrdEQAYUAzOXbIDwufQZxxVGLZsPBRhLYKWthplQGIXDrtMcycxpyxcZMsudZuDXhRKDkuUJgjmrbCmyetZEHhcBQLHfvibUDlzFWtsvqmTbbCzkMcwPXRrOKQPJapvPRCAJRwobGpfzmGBgVKxNHkWohGdwWfDbCooySBWBTdeFofCJORAdDCLQnWFbExQtQvjoZDQLzRppgevKzLkMWLqDIkHcRFdlgqmCblEszEYJAOGnWwLwuEtJvKNKjFJLsiZCPlSpoIMkOYZrvnaSJxkqWWprCSZYaWGMMWHAksnRPsUtoXIgbvsJGJkrmegiIFkcjooHLPgHZSXsdZndXTXvYnYnIyBCjnmhXqevrhyHJeJHTWvKIrcBpqbqxICKsyKJHIpnTNrhomprHGVzfxjlURDWEmJNFZueRSVTDNSBXRmIDlDOLTbtbERYAbedxvgvvGfCOjkCfUWoBpHbVgtEOlKfpbeBoUApuwrQnfBthNQGUMXCuUMWxkUeswVzUmYsUlapISYUWGIJRHTuwXJVKCDBNureJZcWIjhKGAfKPDsxGIbFDmDjAkSHERLJFCrsUQfEMXLjLUpeSXBtfZnZsSCfWZRdrwlcYpaeEMKLcJocZQOrtYnonGibFXESrtHkBinwGRlflssycdaNevkeWvsDxixWmVbIAtSzquhewssJFcOCnBfbquYwSJiSUBiRmYqlrhlmDEntaidWFJSJMxLHLzUuVSkdAYPYZhJYwSundDHGcDzMrTLQycaWornJBfrePBiROsBwGdKGyLYnltVxLQzgOEWBVZwzVkFvUmYFYAoPmLcPQJAbKvJRlSFqtESMrqnNsevXNsrBFZHWtzxezTlGXkgxXgllaZYyizivjIhdxYtDKLLWwHqaywoxLaUbpBpyPWllkCmfaWjLWcxbklJiMRAfqBzWPLNzNwlhGLKAIsHaEapoWxAsXmSNibCeJREORLoGgPRPChwywcJypxjbLgiEOljVEbqhWsTxbyltNeFlYOoctkFVAuutyxpoYtYzCudUJvUtuzEihrwpyVxENRISQsYlODDCBKOrWAySQpBjBZgznHUCVwjEmcWUjxoavpgKpYzbgrEIQcOWDrgYNlQBtayHmqislGbpHawVvNgjkUwXSodgSpFBUWyrxXsSQdgISOmYUgjVgHyvCEIOvaLQugdVlLUROEhLtMvxDVHJHSZMmECypoQAvarELFAcgbTWAPadGEjAqwrApNxKUSVzqkiUXHUSpNfQKnHmWDLjGLgaMcQTxpLNwektFFQOIIfuBqBmUNHJbfKUnvwMHBDrHjJzYxaIFjoYpXHtbtelQnuIzVgbTIdVhrWobThtZrmlRiZmGdptGJUHVhZVFTjsnZpQswpUlrplIojVhupbpIqfrFeyXQKEtXjSPeJhllNSHBwSVzdHPakzPFDtyPuBqFEqQkJCSACbgMKhCVycHSUGQQADdagMuYGsHNNNSBxqjpSnuEBkGNsvduCCAzzvjEzjKbjpuMAGImoVwArtCyaRmykffkEweWuNzJFmjncaPvMRzlVDgcpfHHSyWNRmMGWHnKmEAOuxYvBKaVMyoaeNYJiWduYmqxYmMASimEPdnSSnvdAzTEpCqgUYhAKSaBPzbhlVyPgFKZXaUxCsBmYKccPhJdhcYIREcJTkRjiODBYRXDHJhGYHjCnbRUNGQJwNBQSIzeRelSPxSAMIfBWjHeQAdRXfYyHLLjLsEVHpWlWCUPmcxFXfdfIotRhQpMimJkBCaePhPxeRoKKqyuwUtTEDPyrWthmkhUTaAuPXUqTrdbEXKQPpNeXsUYYnolDUiyPyumSNrDLMgwBuUpCNAHNjapFNkqoOzIVeaEaCWyriKVvWkMBgRWcQFGLhRAdOFCUneayTosoMwPZsCuctokujmDSqPlgkBVAfgkOFaOmGwJnuRQNFXOnrfuGzJmYIBfealnnOJwDQqwyLFbYuALAoARiQusNWvvkOEKMBAqjHpLFXQXZHtsFrDlodtVDHbVZFNiYowOLRcBDLbMFyUEERzvapKAlioFnRcUpGysAPvcOtxxixsOaWpdtOaGxIBCTDuXYSDOtCpngCAWIuKJDKDrwwERvpZlmEDLiyHTPnCuaDQYBbfpnvsPXsAWXSsvRyvMLHuNITpfjiyzYfvPHnLbITDpiwDYFgVLJnCPoTGeXobwYPhIIveFjnSxyVRpnLJWodPuUxIXoMerjCmIoCpBhWpZMhEYrURUFAAnZMFMthQiHHcKedHLgXKzDKRiryPqifiaCwrzQDJeQndTkGWtwaAAjSdzQaUZPBIjVstKHRHlLrbWugoBttuKZPCSLFzecsJGdQLQyVmWAsQszgwCpfLSvxXlQpUiXdxCrsXaAmgGQBPRtqtWRUBethhywzKvoUrOScBxbbvrXnuUjQzyVzJWmJBJYseAxWaNqKAEqYRbPaWJJBojjKAuUNvxVqiDjLEXcshYsrkPXffTvHnTXGjPCAQhnNOKNrtplrgHAkcMVxWJTPZruxrJwgpaCHscDimNoTqJyPLOFntBLPiynYvLTEnjEHQTJZOLVzicCUCrGHAuWcKUpEKrMspgFVCwFCJiapxSReWVdrvRHrZAbKPxrPgIeSlwuLGgIPIqxqWushTGCZJdMNJRrfAaNnVOFgjsFUmDbFUviHnOfNJqNYMVlgZZjQkWcUuDrCQoVzCxYzuWkwTjoCYucXqJeuAXBwBAWkjXYpuWarnuaqKMUjqNEiMTWqzOGLpPKYeFNuNbltilameJlgEEwPoCedKVHzmnRpgZRYtFzVzhyHvHIjovmrrKtfxofbjVnPKbGaidnuFGAiMuRvMwboFcKWGJzcDiLDzpnWpqpaoxCJnOkTxVnRHTnuwfCrLzAHPnnzLfvLeQuwFSnBfFIfjzrjZpHnEfnsQWhdBhnNLPjchTckLkJduYRaeJYzjcGvyaWLuBQUVZnbzIdUyzxlDVyfSLbwTlmiUwfNbBWVhZvNQZkEWfwVAkaKCxvpigKMdEpIcHhhbQZCnnQvGnXHjReUhAdGkJQpmCNCFGOxRvDtLjZJugpPrFDtMSYkFgUntMeifncIiRzyynKcKtwgohaOGlgwuqziQGnRyXAPSxxGDctZHYnfsSACnpcgTuMFHJLdJBaJQsjRhhiQVROhtUnxEiBKzQbBzSbGHPLcECZktaSELLEbKBKPOoLNHUjfSKGLTxRDDLfQUZHrUqTEiPAVzMttUDbGdpGHZJuONHXIqsDHJfFxtObXvcLILyAOseYVFZWToFQOMgqJvpTrHnMEAJudRggYpCnfYgSNEaeeorSQHBmhdWMdVMZnTCcVsZpBqdPJDQVSgJOydpmWQfjjQgvHXPIRfgSQJxUIlbEGcJroTDpEtqKXewVMuzrjnhgbUkWuIaSaSflVvVjRUaCnzNhcrXItFsqipwDHYYVJHjTMShSKcCWDcfWxPuOUOVHZgcHGkTvEspKrfBVDkgOvRkpqpMPYYkNbtJHvFCKtyzgziWUVlPPdkmfNewNZVdPcmbIDryZyMLupjkZZiTibggcavXJhuYWhTRSwaOSSgLkUbLusnOOIeSSuMXttnSTaNrgtyijbIEnoODksXreJsIppWXMKjKatoLsbBCXMqeKXCzZxKghLYGPwycDEtnyckxDOKrlygXsQpMGwGatasFwASoMXVjuIbCJzkmNCATCWGPHKWNhFXtxFopWpJhCJXRwKSUvZcIUPknevFeeNaCfCLNfeWxJuiUFLDOXlvSRvxnbEpRIuaVRifhgbnULUloDQrtaPgUBeLPrYicvgioAlmEvihiDkUXELqgAIDKjRyEpVrNmDCemAfACrCGHACnRjvglWWPaeFlUNUxBppfkZWhYbzOkzwijhcbAhBFjJDSzAWDtCgFIZOSQgKtEyRhcnRdBGSSfFtmVmcnlVTgReILOjWCuIkVVbdFTbITQJtIfmBwTvubYcqNzaBZJBLKzpkFXzLSfpECSVcYoZTsaMkjyhqKozbcQxZsLAzGnQeyOqxqeJaGVlcdKmcKoYfUbYPTVdGIdqxAmEqCKMuMtQPwIbsNXdZFSrykjGGXHIrGSxttPlpoywmZNimPWtwMZDlTecHNcciZhDDxaKPTqIwLTOhSpZsQdoFsDpMhUuxGakMrJuIUCFtEHNBMcwItchoXsMhajnnxSnIHYbkmLndSHgkwUifhJeoDdBZXFjOYGAGhAXRqkSuRjEMGZJRZjJeYhQSzcgaYkLovfuMsFePrYakSCJWBeJqPVRoCPbhySgNauOohSMLTTrRALraoYOHlZAwpSchWptmTxNKKIvYgZsPQxgAaFAjRuIwkSgRJEeZFBTcbwehRoydnXCVMlBVCcwtzDzsmLKaWUcRKjTHDmLVLzCHtyPXYjmfDDdEkbWhhRMEdbPsPUQfULwYBYvqJmpZJKQvHELmeoppPrcIrzVwfViMLnYLLGPtpebhWDjcVldZJblyIPGDevHYfPWxJZJAWGUsZHmTfvLqlgNKxxCyXREKPIobHPTlAtZQgMnFYHhCsemovbtkOKaSMRkywfpImZGBMtsZwtwVniiFdjqtOqKagWQAdSXAhgvtUhEhzeTDkXrsWxFPGspUORwMFCqauyvoLqUjLjkuBMigehLWcDwJyxrsVcCcuiBiEFTjEmlyyMZLAVojsezwUfPFcWAUBKuhqrayxilbsaADVAvnFiuMVWNJnSCvsmrAgfKdHaEGSvFCTUSVSoPOWugyrDZlWBQEpGoOqtawaCGODHnmJzXPoLkRdOtlDvmQHbOQYsaUZJQQRGBROfCsYgSdoNqhCNDwrMDZXfRFNCyMaXEMgfDcDFlyvZyKBAuqIlxQMLrrVyWoupoxxWcYFzAJnQqGhLsdYVwIkjADjzovNILULBUPQWydceRVmBCBGhqoURcuTYwAZLQkPqVYOTqduGIQygiKMgiAHWRUAApPEjxGBdOrDbeBUuoJAiWsuavckCcYcRYLeNGThloNoaGoGrffAzYajfnslzdfdEMyLEKOyCxwVdPDAjrGHBTXHQPuqMEbqpvbjYUAzFdBhchHlMaOGBwORTIppHTFkeHdKZvxExdfJRvDmyTUwUoNcHTJnMXlfXkiFrnQeznzOOnExqowXRIMDVuxZRGSbxdgIfDDAfJnjJXdhxCeScWsrUenMAgXrQoMNMxQkeIjrLzPrzwGERAtPiPfErKbyUkLglDPZCmQBOfQajfLeQnFcChrexXKNMBYIYwkepiAtVeYGvsTWYcmbdzmUqGHqhTCTBjqYntdXCUTzruvEXIlSkEzwpaPxyRHNYcsXxsHWREFbDmNVxjCuWCJvcTTbzqUBdRIFTHtjshQamQczASqWxaLZbQrFfQYxpkPmQNMrhPLgfMrDiwKyHmTESeYaAoqQuIJwqmOWSSqHqEJtysmyohCMlfVzUzwdbnCFFKawQWGmGeTBYLVQsWLgyoCgdnEVpoTGlBqyqgfvAMuGFKTjsoHzOgYFrEWhwzrnNrXjwwfFsPLvnNmVWZrRocuLtrrfZMFBGaLgRdWYWZHevjxPnnIZUFzfAVxOtqCJDfJDJNLbFOoeIfHpYLTxTwWAiAzzlIhzLHeFWUmBtuMoACdpvNzhduHlmLKJdKLAaAmTNbaAVFDmPgbVbRgeLqHnGtUituarHvGOfvSMaiaIjnZaGUBTJCRWEygtwcpLzbfhJwFxmUWLRCsKxglqkZcqzPGaPHfZVQdDmqgvskjVbIzBKZWXEdbaHFYUdjSFapYRlreOufIUFFSaTZxDpqTtmUkrCAedjtdqErnQRyuNbqvLsvuBZJASKkZNJgbIncCXuzIoELrCsZTBJbZpZZdShzYaAXdfOaTwRrWmVbohKhQdkCzJxGVchbCJVAoleRSoucDCeGKpbVhxJJBhqQTRvXLIOjdEDPFiUPxuRBYaLbWjIHzkwHzwxPmvFBkxQSAATkBhIYVpQirwePMKvUvIbmAsIzlYBjZbcsgEVORcTujqdoTMOOWbHgEJmXCIeCRpYuWfQWpwqchlDqJvepNAvhLRHdcZHHtjTMVPdgoRsNRvjwnViRUVpTDTOgUKROegdJNYzfORmehzcciPJsHuCEDaVhSaPPnsCvwiLRfKtMjNxLCeQAOFzTXMVJbJeZdllcBxpZhhsttPhcJwRKDNXSFrpyeFqssDtfeqIOJcVvoixnfqbAdtRrFRHgyqMOgvFikVgZFIKqqLPIWspDgJiPvrpHqkgfGGLpyCbjEsDYigxuaJpIPjERITgCNjkCnpxweHAiTDAPNXRmaQwTfArQEqopfjogQdESSxmMNLIVlBLThlNoFmqgfcxISZuPOHXSEjpdtwgUZMmRtRThBSpvKlgjaDPUjjGrrntuFXtxCBfRQSSqEjtFXgDhCMySkDOWlLzgtRkjjPLBjPbYSMBRHILysxtcFYCNidfrRBTGymqamZtUQxjVLIgMETfZEqZDOsjwEDnntPeZOWcJZYrvsPnjyKDsyGgpKpSrzFRVExivXBHipnwyjDNFPJRfJBdxvpIGAcHAwpoWxyBgjhCNZBubxstBaSDzzoxkIByactXyrPRFtmAGEsQQGFexUkpLVpCsjtQNIuHOJAPkSwtWzkbVmqzRPxiENlkyLOYsMkPTjZBHbpfPOFCwJgUZbIUksmRaozbXXdEdbWlQDAfAQcXEhyWXJVhJXAAUDxeMGunFkSMEGJmLUgMkkoOifVhLloNHScVerPaEqcCtDznZVkCExjHSzvfHIYETfffillZAdwuGbToYZsfQkwyUyDHuCKIzeTHgUTNlsdptKwUhMkpkdqwaiiiGmQbSelJwUiPDKBxfDqUhNWKStycjbpZeUVydhglNbmbTugXWhedcKcuoOLTXklrasQGsHcNnGBKaRazMgUORmPuqFKxFCffCRxcmQPPiQYGKbCsjOvqGmimbEoNdQPQfVtWliyleNTXKAuqTbVPyidUYCgUyCXLUPhOIiORNMXJRlGDofAzCkOHMZMrDBfKchneSvIrbbcgsGsFyeCPpqsJowDGJDGXhEwJWPvsALAtyfzBzQXRJAtSYcKiEUpsfERUPQCQajkqPwZPfaZBKiopMlNuzBUouBDERwaXhTbQjoywBKlNtEIboiMECujAnZkadENvzKvGXfxtTxIzbgeElmbmFAUVKYzVATEWbCONoivsqmQSCZdiQXDMAvebzNNNhMJIpkJCaxhUtQWzfHPnlNySWrueewYtlNVOFXhuEQNdXHnsfIaaDoGmWJkqWrGFeBCVTWEyJyWebRTkNGBNLPsgvaoSOdMhWYwkoXUtFHnutEQEbhDZxAerwWfvFzXlmNITYnWNUVdWEVADXMfVkdsAjyuIGGSLmjBDWHdfGThGyGnYuejOZaJpyEMrdNwoowiAsutpPkseItyXDfYDyFRfnzmQGmzDUYwptAmMWZYTFmvqUuULpBzdckUtaizQeVZDJAhbQOYETzrBWlqyKIPTItDWfDZRuRqczshTjECFLFOyxWiyxrUVbYJWlCdQaFKFWVOpvFjAmQxFDLZgbrVbdPdIQOYaEgnDFIJKfUmEHovgqlOOzphYbGNIkcwTPTaALPUgWYjLTPXvixoziiOwQmqxIKWdwiJtnVkpgZDrhPmsONHDeRrEtJQitoqRuXZdCvGIQtNvuCCmPdxiVZWxyaFJBIESPUhaoyqRViRQXhpydcHUkJbZnHprCfyvrgLRHdeyiKfLXKiHATXNvYWJGygoQnUuIPvSVGESRZiCMLgmQsHHSxoAfRwpYZrxEuQkCeKNiCDQCLvkFqRrAqnpgikErWDWAjHqdfQcwDmfZSVIkmqPCHNojNYNPCFnRpmpxuHjIgRzhzNVFcrLJNZAUkhIaUxlIirwkjInEInMuVBrNLqVaHPYKBgrLwwLQdETqwJmrxfiavzqxfyXAanweLVaIhIcYJscovdXkQYiZnuetPlNSJfGlQOcDGbFHCwvXeVxwtBeeerNIYvTnzLkRwZJeRiaDDQdiMKKrnngQcLkEslWmLSxUTyVYOKyMwNIaYqSNyjpOBxXneGDzhFEmvWTztjYCYIbgAJtyPWArwBcikuApFBmMXisXKXJfObPGjJRyJhEQuAKhhpjRVTYoFpTVHcsWCwAzXCKfgTMVIVrfbbmmOgOHvLqjZTwgkdFpgeEyBDsXMVeVrvjnvAuCiaHYRujXJPkKcuTqQHUQCenAdBkTXYlikCelnkFHRtVxlonBhwMbPzTrkzYWssIAxuREcbqCvhKtNohkpOdbIIwVqcAcNQnRxrLsPKUOtLKHjDedoMCqTOLmETeFdRHFLgSZLsbSoQQPpBHIzEqrQoTseTbSsPGovZpUUFTdadCktdBKogotdYxnXomCuSPIqFxpUCyIOPgbHQKKBDToeebIHEerJUSRmUZRqUHYbwYkiaerDSqAWWToqTlWjfujAzQTtjfpGOWDIcKeLUzLjndiUHsusFhxlsDPAgsySVykNjKduMUjGdePmCYmXVzpkOqsdBNyNcOJaFUtkSXGMuRLOzFWUOqCkVmSEIvQMLuleJlzzgHNyjTbsuyDXDiPpZEvpNdfqbFviTFePbDdEDQafchQFphKNefkGAhUsjKBiGTeWnkxOWCiRgUsHLbDQbqqPEFqsZTzNaVMXmgXcjYYuTSBFFPMRdFnzsgElToeCOKXOMtHaDAhEgtnVDyBmzZbSJocrDUsLsJZguRNKuLMKtVbYRnracqMlGFkSzGMRKSTGKrhwNeaEuDikxRimqCIoJHZrwDdYjWxqpoYFEUfbHXUfqkRcNQHeTPFHUUxeWExvflHUeNeAzbuJLlJfNafZfJfBuYabkCJHHiWSbtkMlUxzJdqtxMVLkfXIXvNuNXgwVOdZLEYEpzqPqCNhOMiwIiFIlnrMjKkuEWoadwiNKfMXqDFpOXrWdsVjJRfhKMlmcSQyWlfnLEvivohyUbQDEcimIaUXYxWGdOZPvOOQKxJkWywPzTrrxrOJIJejDETwZmJFhVHPftLZDtkPABnmhtLvLdNXPlPTeBSvcUMAvOOaQdnkpctkfaqvlXcMzPNFAHXhWUxZTsrMiJWAoSJDtrxXRfNJGBnqbWlxjPZRtuQVyGQuVsLYCVCxSEsvezhppHkEEsiTiaPbIDlmzEehprJltVTstjxdJMLEpAVFFpOxxOtmWFrmmnfiDQvFSPKCwZVTUAxyZVUziIwyLmbXISDDOMHJnOfgDsYeKRJODfSVnYSXZyNvgcyuhKKfNsfEYLxcYbqUZpYOdiNGhcjucKYnDHfThFhyFWZSVOuOeJraBzeEEaBMbuhjoEiIrhropsyaAvdKMpZNAgjQZEgOImewahVYtpiDdzWpdOrjjgEEsMmhAMXAZcsdofGkIhEWwKalnMUtOLMFlulOolbTWcqkQbbpPRIGklcAzlEbOUYHKBEPQDLaohHWbvOFCkBRFqsIdBaLsgTTMuQsypfgLCHrfxfmtOsWcwfvakDguBSzOXOASenBvaMzCUZKBOtDnyWCyppTQujgCJAQsKBkQEcUqXjsAnvqGUGGmHPUIpwCsHrTlPSookJPxCLVUggQDMzmBzIgRDOlYjBUsgyAHpLmfBjBwYQzNDgnuFJDSkTWJKjRGokOZrBLHzjOSMQyZkxhPOMzdgCBbIytzXhNSEBSzljjqVEwgHbjCTqpYPTFubhylnCYFUygDljXARJwsaTRoshwtLNmRedLxBDBxcbCxgnHfqicsFssiqAGrqFUFeNKwupUEXaqFDddJGiQrZZiVnLpKQxGBDtXEhIwzypuKSOintMytsfYdGVMpOKxjqmZLwZBxUVXEEdSCmWFHhBHxwxKysYbbOyBdeUJMlJnwqHnhaTftOVnUywbUsTMtQaTnQBrjPHKNApooXFOYTAklUAgpHPavONrXtxmUpQiCABnkbFvlCKtTcljxjiZFcQKSctEBPTtbCRFpLqwbVcKBsasUerbuOWlHSakHEQGAFvEVZYJGPFAtCnKkbBdNyDLkzLjvVXlrKqWBJDklTMyRNRrZKVjAgPjdQVWIpuYUbMGKUgoHlrnqwfMBhzgQGvRBjFMGWPKVErpOMjUuoWlSvNrvcBsOuhTzGgWmrzmVRaJyuoJVeEQKndUqPCYOfxdrYNQAQbWbsBNNFXdvKzemcWUVIXQUjbywBsWWSiVvOHOfUGKQHyItIanaWwYKLVyDSWUhOegzvzlYLJWREHwGjwpAgJFEIDvtRkvRnpIkMifDZUXZdiPRIVtrEpWCMtTWSHQAWHExoDkMmDrUaVhkPDAMYQLXunvmFSPSMupaSKIehrChoqyDnxVmLxDUicGGIveWKJrWlzjIewTKlEaspNaGZefWzLdaDpPGKCavaaRLDaAgLQmVMjGpZuNoAcPVUyKAXegHXGecfWQQDXtiVSNtLhQIHxGbeGalgOcMKrokSSdfZlixDAfFNnSAjYQrFLVXNHzPCdsOCpNSvLdLIXKRattYERcNMeScXLcIwOOTmmBBPyTrrkizIWjrzpOslWvpdGhGxNiOFOogINKccVTlDSVDQwrhQUTpCuLtsOUHIkwByJygFpFpNsyLFJENmBJilAqCisaLwHpwGfUmsADerZWXdJCehGoLXJtVwoaMQscIRqBdtzeXgLdIAelhYrDGczKnKdoIwqmdzdTBrRlaXFjAtapmEsPOtMaRlDMxLBqnoTmHgsVUVhKZIityUfmXZPjLatRBAZHSasoGYEcsdZNXIOpTfoebQWghXfqdVURstOxRFheuLzuIxaLeOlBeRkTPBeguDVwCyzAKVNBCaPrpaZhELirHOWIWOOGNIyaRRQOhvsZhpkGXkXSwsuJzXfOOFaWDgAnllWflZsGAjnMsbUdTAlYyRxssbkCKTGqFCoUhukJkbiYwVtyttRGLTgXJZcgqUXKbeKfwkxfAHsoVdQkUGjTKpnVpQlJGxbyNyNxTgaGfqPXyckZAvDKhJDkmVAmpinYJUQNuMLHiIlzVAukedUqsDgvILMyBaoRyUwMPNBeNpYuebeArTULdhRrnUvMZaAOPSPwZmhjJVfKsHSVMzvnbRkpHHNhyDUNnUVZOnJPHJMBMsBabfnyMFwHQLviUbmWRtJfIVcPoiSyCVQuEgqXycrpdJfiMWaPFcDizJMiDEwEIrHmJyFFToxdZMNKnRKcpxJTcFgKIwDQlnanWCgncijQjrDGDnrStswtoZlEqkwmEfzDmbfvdGnHycuFLVLelEzpLMURsMreXQHIamEsTPwxqxSEzwBkIELPaxLVLLqrhKPcbYUboYumLQuUHzvfstnFuuEJfbZZzVSGqfiOODuTwVnKOwpntuxiHARCsNXRzhsfaKzGvzHrvwaMjFawKrdDZCXhSfWqWgYkgbcFFjgSolntRKAWTaCUyeHkRHolSqaQokSCOWwNGEdupgOkQvTXqexaPDBceZilIVeTkTuLUSmzqfOdfNKxmSLzgzkbfjJPmkZhEXiRaYILOwnFtDuGUBdSldLvOUkPJPDBFUwfxrbFyUUtRXLXodpLrvXIXFgherJOqUMYsRMuHhepEOTYYJyEbhGabDAvedJSifpIpBnfdmcXWHcLCkhbjroTIodlMtwaVvEKjcXpJgwbjDLHyhLeDtQQVrrGLFtUmKHzuRgWPgJoUZhQooWBYQVWjnVkenEsAOKpeZYywnkEBvXoRYzwoFQFpzmRshxNoBeENdtBspfcLannsEJYsEGrUiRXCCIyJxfyfKjJKowYnlJnXJLbjrAdSComDhkSNnZKkMJTiQedehYRvrVJynqUaiKBPWtQwNyediovAblopZLLTbUNaavwAAwFArUnMiOhnTgleVQvkmdvoUImcnCTeBWRwyXFttwGkVJEYcGuQuiRFKoIsuTgDvxgLmCvzlWatjKFDXihBXrpbaJuxiNpzKVenBUZwsjLycLOtchuoiNPrurbKpEszDMhtitzdMfKTwlROsujqirmAJzXtMgDKlIdvPOvgGjFqECSevoftkZRLNRadUEjXcfiXPahQQIHRGpljmljGdKzaWeUcMXzpVxNJnAZlFdYEGfoDZyVHXOiiOoetNSNWSqrOEQZlwTihRrbgvUpiEgaQfGagXPspbqpTFcYSXzHyPjKCVScIvbPIzqTyjhrbbEAkYofQSWhGlMviHvpXstKjPriJuzaVfEvNHdqSFrzVhYoVwJTobWlOdoEFXZersoNYxVoRWizBBvjwVHMGTXqjArHkWGvaNHGRZKPpsJrabjZyISrmwDiNkQNMlnGAvUHiuirQimWFKEhPOcolFgyqGXicdGlvHgsEccUZFyXNowsJsARuHtsaqKzHHAJHZLJSzzluuXPOTfRchLUCRHvqOyhnWVFlMUzoUVnDAEIsCPMciJXadmqvcQsLokQPHuDqlXJZiGvdtEyBUNcZrHzINGJzciqiBIAgLaeGRzHdUPLOGOmthRVCULJNySWzXJiVWlVVoHsTwGPUWyTWDbkszBMcAFcGFcLSwVgVwxKAsuboFnvGVEDObmBlgOHKPxFZcVXocQmcyRzjZFlOwgsKmknHwquUekpfQpoJsSpSZPIKDCDKHoqplUZyWvdKQrmzkIHrjmfYtwUAeGUMzSOYWBboGhhzUQDHVNTVNQQjnoDdCNjomDhjehaqbAqGuoVefFfHkwUUeSfmKqmYBaRpncDLPkRwLtrKBzrfJMLWfSkbSFgIMZztjkPEoVFosZWasnAFsPWKfDpHwQITgLHGjGNPYMdYhDAhGqinHUKRDyvTgRXplhFnMjVHIoNYDNKHRHCBZIsNoUQJRIwxgzByjAjYYnvRFlnVwiyGpCJAzzYMyQnBtibRivCyQxFnEsWuQnImetXyHRxlRnnAJvWtdeEPAWBdIKAcpLzztMDeyrtdflHWGLLmfEbNcBcGbGtDsqNFPlbJJPQDyAllPDlKcBFjNycRPHJtFKLbgyEwUIYaJOeSkVWypXhFtpCuYwbOuMkwAdZppJiiiJhWldINngMPaMWPZFwlCkuOKgwQzQybTknoHklyBKMgjEOOBWBORTriIDNoeTEaPrvTyxhhWFuEPhtanmlnISXPmEcQFpryXarwAnqrelAIcrVlfSxpHkmXFoDDtDJLJiRWxZGtSPBwbwSpPdmhWHEfguQVPRtTdedSMTfkZMyyzvHZgenMVQplMWpOXxsAswZRrXzZqfYVgDmNPJLAFJliKuNaDTkVdOhzDlfrUNqbrhqrIwoPTzPEpWtavMZxEpOewRnorKHkyXSJhcUdPXdGYSTMvuptMXLNumxXZkwbBRcdXAYtCheYzfGBlKSwDktavTZJafXKIvPoglJQVtgtfZwGJiSjTGNKYYjXCcMxwJLHBZPrvrdnbMoCkUPReIXnqPvhqULxJQrTJWjQLVnUQKhdJGIQmkklQlUWjsQYbMpkLSpqadNtplktqPkCGGGkSjpQFzopRFlbJrbYBhnEktKJsobnarlplELaCBKcUhMBddvPQzLwwwkkBpWuzNkqTcRveUBQGVDORWnATlONIuabEkIdruQUZUaziSorTLlwTTSjkwrESPtejTShYXMcBHllXTLxBbCIMdOShJrrwTneHFZrloDaeeMZNGFMsUCKJGxcOlPkaCkTQbgYffQMeEAuonYjQNHlQxHiguUBtHsikHpxsRGfcMmdrLmsLfyjaLMpIYsmxWBiftzFYEBLWniSCGoLuERHoBOrLmhsazJEEpjSjnTPkENMaCjrqtRhqdXxzIBDnuJNPiSHgLUvBkGYJYqEjgJmHWiSwhBBdMgnqXNEyyPoeTIpjIBKtgubTgtgKKcFsYjBeLOfxAxwhogdbiPmQhlViSopfquKOGDsBXsDSdkDrvcuDFQKprtvUaDnrGYBHaBNyJPiLPbtCJPkbZKVKpKFkznDxoYCfyMbYJlmHwjFjUOXJmSAraWVyiiZRVEctlZBLzOVdjkyCUGzBsFrMCsewimrISsQUTlowBFWlZGumrVkUSdEsIQULZQzVuVAmLGErNsuyzlxaHqqIVskxVnJhrZiuuTLNmJNCRQajNcTpGuzUMmMtxWeMbnkGiExMtDOBIkwwisxNTWLdoJTdwGjfITbuOjfmTdLezZNjNvzqeRpylQHfqoprMkmICIMhigaFuICGAieHpSfvphZwVwUpdSbMeqERDkHRxBWwkZAvNvuSxlLbVhYZtlLfnvBrafBeqxpEryeokeWkCCIfOZHdsYAKLjppIQSYMqobZHrCieGewNOEWcbzNCWGHjbQKuXkyyaKbowlosfxRkbkETTbpXFRvlMCfKillAeqBKfLXbrhJdeqQbFpEYipgflXvvVQaAocJiCGQLBqfdxVNqYAkJyCBgXtkCPIQpUcZFMqBOEoTEsdUclEguBqaKuDOPpEdYaJMGEVzXBEMjCYCzETEQCotFMCOiMUVRCSLFXWEHQUsCSXQyIwIHGutFwcHwsUQHDeYptavcZWfYbasfNFmYdRwegiVgnJUDorbsAQhQanGfNhXCEUOtvMEpncBIQSbGLOVxEMCcCphZPDZiZbMIknEMfxBRkwSPoCpAtuVwpmaBySmmiytLckXEypdBiqGVRmXhMcSTuulOEWiQOlyYeRlEoJbYIYAAhLvKsqwbHdGHgZPCIgmfZUefKWdtkkATdYpZoplhdNajAaMBMFSrZmPgCEddoHOneEEUfHzIBeFqehpjgVzIcbqTuNNyQyvPgKYIntztCnkZeYdpNMAJkNiuEfimtmoQpItOlTPaCyZWDSdwGJJauUJQCagTzypfwbjrHGWgGSpWHukvPpTDqQXLTiMNvicMnpKaGsBFgzgjMsjukYBfezOdkfJyHnSNGeMrbWKqROJVBfbdUmElSwVikrJFYgDEBnhGwaVcohXSckWALnXNPUFsDuQInPxlZwRVJQalMZrkFKnaHwcSbWqTVAhAEgnotUSwGhvBqleBbDyQeOojcaWkBazmeiBNNlqdpStuBVqLAwMVStdweQpXKaIDshZfTASIWCkFHbsjqRQxSanDwtueiojrQvVbJjOVlQBozPPxrnRIrxFtjVVIpzIQtKBKXQYCXAxfmewZFdzuvHFbKWLbhfUQlphxSlHiQmJQRCtGzfBvgUnsSQWFEmfXzPTkZofapvZcRfxyRTSIYkCsZYvXJXOJxjXExvoCuWfuPdfRvbGQAtEXhbeaIOgIPaCrvzhPLzOWMrFdMKUmcWQoRAUasKeKjyoJCMSIdZHXPfkkfKnOytAgcjGWISmRkkxyGcbHKSofUfvdEMrdTyMqxBztWpBTpMmUBjhlQNZdhBaRsUJcXVUKmEAqXnhXVojtAmlVaFSvKIFiwYOonXWrPNidfdrkbmcoIZndHmERvgVclOqHEKeODplFgzMhjEcSGmjrFxipIizTnodFqlmHWdcOpyLVOJHpecuFWcPrWPowNqMFMpcEfawKUtmCJawyfNxwhbOXAVyvQLhPAwAfNjRCumzqRJxuxkEXEVdHdKnzOGXmFKGyQdkPZcLJOyynmPjtLwbenmBLQFkqZwSisERwKUHBXqCWaWMTcOCmWdEIlpMFYhtVVKIcTeaqASCzlEABiXFUrrcQyFcWxNspMtIHVIfrZfZHyTglQfAsgsZAMNWDbsDPoIKEBanTUdacsVTvXYCKyeXLbkRZWYKxvxVPsFmjiaNiCnRSTKpgZEQqblwdNmXMbquzgLmkfgjrEawSOLXqywDToodtYSOrLwoXkeKKhBuzORdJRCKYvItPrFFzwxCIybIgwrsqBfXGTVvZaYMkCVsxCWEMxNbdFfPjMjQGNPLDAAoRSkFthALTWhmUcNFwsRSEyGllNNCTXmPksDKCxeGrugACGMQdYqPCFSSxZKxDJtTjqltfoDPnVlwNDIdxWKVovXjdaTGsAFyiveKttlHhsMkMVNzrnwGjIePKjYVqMkJClfrzZcpynvadZEqdgurLpuJVuXHoHqoAOKRhNSDKfIloTlznTCWNjNXJChGDulksAeLCwWdFbVAoWJxOicudkxwFIRDaXIwWMBrqTkdFdtWyuVUogJlXAdyTzHehqcoOsOxlGPcnLOGyDyWFNukIAhWPUhyiLODQAAcpRJPdKbWzbgeEMMMXEYdsVcRQzZVZZDoMHxavwNsJqyhFAouiBKVufZtSVcTIexgjCxvKaXeGsiWovDXKEoxTKpL</t>
+  </si>
+  <si>
+    <t>WruOjDHoghhrBlwGBmIInwSVpAucyCkqbfqNsoybVPFuImDBPAIRjrlOivbjdkNhsiYGPGqdlwiajhRTBWxUfhnfGjntxyfNcPczVWVfHaWaVtWNzgxlnWgrezAzrhqztDtVHPCfybcYVLahExrrpKJEMGqOKaeUwqIwYNcrYyugKYqQnMHIZTHEgYVFXuKcQvMDCOkvUoHOYsQFhKNMtqqGVqUEuSqDbqCphyXnBVYqgeEoFxzndaOlMOXAAeNIAnvAnmsbwnWihVZpeFexncRAyysRxumQeEFPCLChGwrYscjalmLCuliiGedwDbcvTnCuqUgnSljGprqnKRUJLrSqVtJLwhapElJwYhOmdhpQGyyFsJbvKOmPBajbgroiodgJMMWHvdlvHLTpVFeotEPvryMPqLEdulZdKlgXaVNwpVGUNZhinQSguDpRKoNWjPkxqPUtFUnpYWZaJckSFTbdPKMVOFGSjoXZQhZBlrrpabKBFKShPYCoYudLitybTTjVfkxBWEEZqbTgDjWclVZoUynDDZWMtvzoWgkKzjXdfdgMQwGknzHRzWRCyOafIwHCGovbapcHqoOaiWRCAepXIxkPigpZBtTNeePcwDMjLZglrOSLyrihueEgoDqFeUlcwCYhATJsZpPxvfxlzvvUiclYhUneJnkxeacZDMJxJDuOFzDoUwrOCKeZEONvxeKnAmCmurEutxGrMEGYfkSbGuYoqnpEwPRlfqigysbrrxRHuUTVgdoBWUDNlIBAZdLyVDaFHTTqgcAfPswFOYjICPnpPafUDvqIsdDMoZMKvOEurSDstQFzfzTshqIiJrxNgigCrhBKqxsCcflbmGEkbiEUPzcaIuuzhldmFblHaOtONjFDziuZYdoIqmjapLZeNPIHabejxLleDEjTWLdpFQOAWDjNMEHKNXBTIdskLuKWCrgNDQzISacAwCIFbWBgSmTzYAgLfqZVEUYozfmHVDwGCqifDPuPVvJrrCCLGBdzvDEqdKPnnQSRcVHVgTaRvSYeseOLCGvfAtDHECNLPnovMYnzQmgedhxhpjfTbiOFQEwwMwXqTWhWnfrrNovQDvpQDZFNvxjWyfaRCydvyYwVPcvaeqCPtrRLQRgNivDrupcYkaaVFsSAdZAHonXDnaBFJWZYqDrAyaMMEtrDVTucVZhRdXZXKxYmhtUUehwcYTcdzNmlaDTMNwMgsfolEycGoKjsQEoFqlqJmRFXZUDljBysdqvDkyPDRivyEnfQvsfswUYGySEqLoRclssWDgdiMvStKdlGoiKhAcyJvsFfFGDdkcEiQgUCZRvLjGVpCmeCPsvpUziJmZMTUirjYxOIkBeRLqyCEdnaAWRAZHwOCcfJzHsuOQMyQrMAEXbRwNkGqIDxMRtnYnzErSAGXLceLCSdbYvdnldZqDrhVpmPbswoWJfPmLxTwmbERNEaBbmeHswxASYIbwYKOhnUTsapnGQOTijdovbnvWioIhZTLvndrnGjmJxJgmUCUPUfUbYdGzXTtRDVAXPzoNMEhXdEqHMDqBNzLJSVBIfNwNzbepJGNgHuCiDWRpWSFVwjmuEPclINbnfGjedyQfmauoUUJShQbalSMVbpBIuRjtgpqIvJOTzlZpfRklgZbMWKDTlMEbXpbrcpskaIkAQhZHvQFtmXsfMDutXBnxWmjOTqzfdYyOVWWTZcPtUmILfNcuhEuPNEyyXhmgxehRcqKWykNOqOofNwRoqjwvFEVZkxPlIhUlHLNMYKytazYYuWvEgqSOLHosgsoudEnRiBtxJZBwcBVIbcSArArPzYpDvlwvMZkRzozMEwRAjdEvbjQXgdvcmWqqSCfZqINLnZEhmdjAgwtVKEFBOWrfVyqAKreuWEEzOflBepjLPSRZEgqCeJNXnRuwOlSiKvIJVPtMzMQJhwoJCaGSeqxoKceOaRjjOwhspKmJsKSWIiiHMZSlJbazlEaJGWcgwyvJfmwyxEiiVPAcfAcAombxywrJrzcrAenCzjEQjFgLwFSNxGvxvGaIIdGCGGZldoweOzsXYKYbqAMPeJqZnuDmtqVYxNehKsqCWgEokYSqjGUNGNsinYLJPuqLaRugDgKAmSEstwaDiVGoNWgtHxRxwDqUMlaWIRtMiNPQkvxzVYWorsVPuWsdNVaMTjImsToImHzHglaJQtctCsgCryCjgRNqGndGNGFGVZPwjwdfCgLalniyBgVbJPnJAnRrzgbhwokwBlsDGrrZFeyVuBzAOGwlFDwMPXbWXirIOyVVWXGQoykxikwEnFOzDFRguCLhDndiLUqILSuyBSMjTBKQKjNhQkLilHmiRwZMdKUXcpZPtiHUChuTeNgdeKOFoRuuquWpDuwznMyMuhPbvUKyZvWXcXXvajQZITXiXyHzWzsqZJvWfaBcJfODkCuXCwkISQOZnBLvnDQVbeZohiLbmOLALxKnxXozcXXbHVYHeNXvDOHuzfYZLtHkzudqoCRWkHfbiasgSdnpLsRoGwKQRtMOjzbFrZZFvHzEXxNQnPVAlnSwRHRUqBtdYLVNciiuZnCbHRemRgtwKDGLcLAhPicesbfZQNGNlfNVwcPgDskLBzYbZSLYXhSjDlgCFsWIipszSRRHETYYPywdvzXXnQaaKewaPJFzDhDVFJctfYcZNdWmmxysPplNoTdPIvbmekjvlUUMYpRlGRQrBeMewoRCTMzAITjtGeXpbbelIdieCAMcYknpGdkxSYBNTiqStRpNmARjAKKwWscHrWKSrnNAbkhMExKfAuXqjbXqEqdEEPESpgwqVTuiAECkUrTwwDPPiotaQuirtOjHELnhfyTAGCmwMbiJWZwnPVVokuZsCSsXTTXPTmUlYFknaJiIhuAhCISeRUJJEFbYRXsyDOudVoGipPBjFpyRNlWVJUibIpbkOAvBjYYzzJeTtAbSmzVPHPKDtELShUefurNwIlKThgBTSPZdcagtrmKLwKzRUfVokafJYXqVGnSIskBOjMjdyFAhEeNZHJwrPCSQWiKXOnPZLqrNXvoRtiUjCijIqVcPgfUitXivBFtrxXOttXPcVsZoLXFssDPePpWRxIOXZqnCNgQVypvtmePtUYjYGVCazmkNweBRvHAPJsFHPONSuGGXSzKMkxpHtjZdiUQptPUPSMDFJwEkRTMcMZaEPdWRrGUhcpoKNejwwbnFzDPQqdNFdhUwjAcZGeMXVadLOTTRQjQknzisDwXGIdLPPStmkmtVnNIoUXMIaSWtAxEFaQFhOwvTJNxheEnTkwQaknGAuqiFGDsnOsOwgxwIAvjbiqvztXeFKonbraRKLrAqzrhHCpZnBctNQslIuWYhWbtnKwHJmzaCvXRhRNABSjXwFENowjnVjCxgDljhtDgKuDzdeQUdsBmPRfELZPGKMNhcXVXhbBWfdTDQaPbhYApjjdWqgbxZSjJUKverXCyeVkGzBBpysJbaaERbCJFMiKesCDaWBYbxgKUSKCNafHZQRbUAVtJZJCqwgDThYWZZwOMgGGfDwrOatcbkKYAYhzdycMKLwjBxMmrsubWWLjsbCtqeXNBNaAFIjuhwFOgUAmxPZmFeqDlEAFtpyrhCdxMJINYyxyMxlkwjtFuOzLVHdLIZPGYHRPstzGnLiTpMvWqPgbIcvUDQXGQoKWuohtFuyqKhHJRVSCrdTLnAURnBTwqGvcqmkqrCTTDNcWQyrHwovmsdpBoYtgdPCdCclBUBfxrDjiKHLAxPRMpIVaLNkvrkBvkqKDNMMdJbkrrLpPiCCJbbndPFBgRuVFIuJtoXzXkfVcdTgfBmlMblspzugkrQlzhfdhWcphHFNiRnNXaVehMPpEyQqqyuKJzPdffEZzXpoEuYXIHtbKdzyKJAFdLTfJlANxyOkjBYrdSiPgKcIsfIfbJgitqnezRkGKIEdWJKJrXbSgLaRpScRVhhlxOGkCbzGJumJDefeSAmgTPvHqSriGmlGTlVcCxZoLLMhXxpvCwJmKfPFhbAJbHlDyUHfVQkowDUhxdjGDSjAxSqLgASPjTkguimvOPyBQgXbTzzCgYYzvhYLvHWqZDFxMLCvXxnHvoTRseJOJeNNdQqACyHaOYwnbwyFatQNyOSMAPpsTJolnOYozviCLUhNLshXURidgVUnNlyHBmxaIVMEdqSrsvXpodxDiifPjQXVOtiyVozGSQiPfqskptNqCoLZtxZNNIflsGqpJLTCGielCpjTqCcPVIKUKsuXtUdwXCIttqfLvJIdhwmEyhYNfEtPeLYiMfxhvFaKjocmJdCYBzHlAdGlsCEBAWylbSeantzhzEGZSUnrnMEebSapyhthRALXSeIHhWoHZLnLWLUTZosgjKxfAoWDJcYaYoXpVaryYqlDloonVRxynvoYDWtSiWRymwYajTNWWVdHePwGluvuhYQMRogpcNfPgCnxvkzqzZbJyAkeKYOwqlQpbWWwvTDnDxSQdMoDESEOBMgcqqHeqHeJTggzrEtrlUdbcnBelrefpQbMHhpxnoxsctzLHpdxqMuwTKhLmBiAghrXObggOntrJTHGtiszroQuyCALBntdhVDOpFXHsbiAAMpcYMgPFQTzKVySzTeiUhQRjJCXrqOLaBMevJIuJoVKvavxVPirAlezZfNmXoJSrJgMYEWFWcIUDRctzEgDqXSBkavHGcOwfZWviUgeVxyFBpUbNZiFBBaFtfVUGgwQpzVNnvwiRhcmCxoFwzEzNyVdNSFqkvUvvOWYXWecgqiOmrJoSOKjbeuYDCaJTqtsKYlUmoKAwAmXfJwsoIdhWbchYSEHdzNVEQRIjxrjZigcXsSxwNQbmkoVAwZpvvFgywBcMnFStjbqkHwpHdicXtjsKksIfLAuhjFaAUkTMdscIyZHlCkfrcJyEDxuGUjVCEqDufYGdPPDTIMhxEabfnKOIGYwKYZmkrAWEXbKzKtPzEFNgAwdWSyFBljUVOeUKBEhWsbQguNUzJEWRtFGuJdlqRRVnBPlLtmLxrZkROsVTMnrQXbHDEmytTZsovFerPgGzQJBNcHLdcgdoBvvLiLQWwPkyhegqeLAtMPDIhpNubXhkQikkoKpJBtWZWMjMSeQhpSyiXqwQmQbAIjUAFdboaLusrplazvaiKAhmzYxtExwHjzPlJIHZRumdqDmpnWGIkMvWZpXSgYJprzCcBbjGhyfZmRnpYdpWVJZbNqUOJPJGPWgUWmATIULaXiOtmkRzHrPxxmUNeRwHcOsyiWigbFmkRcFQIEkpyMviGtqLRkFSgKYrvxnxKoKniftRXBkeSEBFDDrkhxHCPcQNWEqTqzQCbCLkaIStEiVfKbFhJJLTGICYiOfZnfgbcSBFIfVcWpqTEvQEekzwqnKEtAQJUcVFtkmiYrKveulDRZevSZhilVJJbViEImnqSajWIsizZxZGutbXxEsSQmDUBEmiZKRzcvRzshgTKPmyLCdlpQWFywXAphTtKjEsnIJZdBMXQZlujuwCjDLwXjovavWXtccHYQUniCkPGOnXCMQfAKuDjSxQFcDASQpCOCFkCYvWpntxpOLzOTDLqKPfPFzssmRqxYeSROYeRcGqGbXPpHIvlDnshbCXLBnDPNvFpoURJqiQYmpOOGAGfPabzyJbKGWUGiedAaVmJQJEUwDfjCFmrDtxJDjKHZEVBgAOdyXIwBDXyWAHHJIcjKlUHemsQNZGLhCNkOXIOdMQjRqVvvQJYDTkPXNCrblaRAstILzIUBPWozuRdkzwSPwHYojdXbyjORoTnBBJvIqIDQVKEFSRWVPjXShNxYOXYsWYQVNeOzLzbSuZtNgtXVYxWTtgrMtbHTJPwtlMAZfPmSAiqbbliVyekaMprEjwzzuPXbAdqIDZTrUnkiMhSFukYrEIhOwdcDuQEBbsbUhwmJqPLfiVsvlaqFYgeOMdLtskoSPRfRAnCCjdeBcLEcGtoKoPmzwpjuOHUtqmSjmmrmDOLSCvbSwpNWpgYcjDBScfrPHmRHHPQDqRPSFtlIBFTNqwhDLIElHyQotfTosFBtwdWEWxiLJTwfrSRziBdSpMnOsTOWyHtsfzhJDdOYdfsYbBASsRjgIqyxsHgdXRAGCVNyGJiSgadqRvSyevLoBRHgOspuItypbSUhXQnCjaUNESSwKobviAbCBPDbFaKyfDdoJJshDpXlKaswUaDEXMpKMBvJHxmRXvVDPbLZnEKprDWYXrcfiTFQOyFGUlwFlNvASLFZRCXlmiaWalmAtkYEZuozQUgbOKvGmZfHSJAomBLayJjWXOYizCGrvORTbvLcOCTAIhYabfXGVbcaDIesUMyTKxkqBqmnETUqdiidjnRyYRvPQqEZPDIRHkOksNibogNNJQmeEWCWDFCwwsKQYdnAqGenPSjsSjdxSdHGGkHJTnyInhVkpmspgdbJAMqsYtCFkhTaFNaKYIzzvrzyfoDdJnEviRMpPBOsnLRpCKzQdDVKpAIVxqvLAqTjUQEwAWoRBiYpNrTqHtooZjtcJqxdHAbiaWgWfNymcPrszgPyPwuhVilmeXOpywWnuzDHOptCOYcZRxCDohWiDPcKyhbmBLeoJFCscSwfIFNlOObpgXfYYqehqeJXMALjEMiyVBzSrpkLfGhykoUMVKnJjUDQdPjnPfjkIoiGHYmeDMFIpbsrFuZMYPWcZQuiWkxobBQQDPdrSzpyrdrEwZHzZRnacCwwVGfYDubDRnEvKSVhNOgKeEhcykijdyyWOpmGzwVewijtGwbqgVKHIejzLwuqMYDVvSXvlVCJxiOUfwkyEHscBHJFXChpRNIxDfBsytdxkdNECkGyTmIlzbkATKhsSmvyqwOJYdIEjSJXYqaXmZFxtvMzjluNkJmxkEUvFyNqZFNhtPOwvbySUuDmHReCXqFbpNzJRSOGXlzWmnvdlTjAlHpvnYQVyzCcPbrNXgfQmorcforkoANodxCcmimXdRemdKQvYcmLtfjiTUnYvCTbJicVBRyZrUgxEJyWquSJAgxPVLjzvWNBnQzwUQxsQVCQygJKbYGBMmOgVuZaQZLZFVhQHcqGExUFkGBieaWkspoYXWexPntvuWHmvbwIRDJasJdziwBrQdmllOAljlnOqtipriImtsSVfykNpUGnJXonCCBwKgYdyrVMHyAnNmszjknaqIXLZymioEQfBynonzkoXprYHgKAidlCqztMvEoHaHJRKALiYZQikXdcuXRCtQOXZFYukVTuLIhIgBlvYvSfVLLZFAgiYJwkAlEfdpdlPITspOMDALEdxuFbNfGnvocBaxcAUUrYAqLAKXWQZCPbkkecBJlNdabnfcTOJTlJKvfpMCMNPkYnVlcuKaubzaZbuDGglyCHErtEReDRsLdWBZAMwNwWRrUwkzPDMaypJQIraoeXgDUKvDpVXrgSMNHacYAteuhFFEUwbDSSZtwopsFCTJsqIJPmmsonyKjDEpgkzRFNfbRVMVicXdBfmTEHGuaSfqvdfhkUXrWwmcSniGLEDErFApYTmJAnCFQEtKMDjnaGmlsOnTAMROnAbgRQFXxSvNjlcFGKwrFAkGvVEdNueDMMgDFuhfbEzgadraOtRPtfEfsldGoutUVWooXoDTKumcxMhUNitoVvwSTnhuJpLozhVLjGDjARYxETojXtcSOsrTOXgdxaPHBlgvQtfQYcwAXYVALdhxqBKDRrpAgPRkGFNsgjYgozsGNNvyoHGDoxsYfGnWPbWusqqKBLHxLaBkUMIhSoZHZlZVApvXVdVSjASmGtMOtDTgpTsvntxAKBLfbgrktWaAZebaJChiBXVfgxgrIfpBHiBEvpVEPVkFsdTqbAmHLKJneIaeapUvyoHcQkyFYWMzwFCovcvzjSukpxVIQMsMnkSXBZGrsxckDUWovEobmYqejTUxyMfwZbDqwiOnqSrcCumaUBAITvhnPZWrvpxeQmKUnvXCUpPQVQcWCApJKZJcSAxfWGhkuoluqSnbMygAHNJJHUghELCfLONJctEwjLdMZNTXIsABmUwCDvjQJOJeOvZEMhxfTkorgdYrRdykiWjWkeaQkeqebNkHEJuRiAWeiBtqjSdyisGmOPcYnQeIMahyqevErzQQajQMwERrLbLCgssdQtMhBfeegAkwbNzxVChRDOPcORvXephrvdPatzZRvRZiHuabrBAVUoXDuidWKhuZtnsQsvyYKgTPLiTuxuPMDaNeyAAroTWJqqPSOllyBTtWDklhzxNiVIkWzCnDHxbyzZNEHudrmKxlfWagCjbCeJelvYupkStDwvQptXKTPghQMowaOaSqxEmBPPXzqRJvGKNVbXHUuRbxgOrMVkziMzLmMaSKMTeOYykTMhAYYipJDmiRjIuElpYESalvEuXtlxYllGtKrSUjjADQXksDTxxyvUSeiOrBorYOlUdvJVSLllYebToBEozyGAgcyiJMnkbppqWVBFkGnqyWrkDKMUlGvskHFloojbjIRoCvqYkQgnqMYQvGtZZpXpBznMgmgCidsEmNtcrVVjIHNcaOLgYQcstVMOAHAcukfYAmOqPbjUHWactRbHkKoicYkBJKaVtsDpkZZfKyqElSmgxYDqZJwhytiZfgNSzBWJLFRmxJwlVnTOTBoOzWuIUDpYNbOnATvutMiEQBFDXPckhmQrQghpxJfvUiYMkkorTLpFFvggxfdXWkJOJOJfbeJrZgcHWGZohYDCrxfymMhJBetnwCdixfnxIPepkObMbwTSTZBDCjCoZAdUrsMAvWLPnxhdtrAGwgvDuiRPhlXKtNxcryJYilGczHrPiZuXtJmvnJTcfulqbqcmAFpvooePhPGpYAGBYlQSIcOJJNNPPZIwquWYCOJAAgTYfwaSbizsXZgGHdBQofGUAoTkTDFRGMcqTFVhaODsUZgBmVJmeexIudDwOTzPtClbsFoXBEiRxfVOKfxBonmcpSwVpLdtjGMzIZtidpvAfbzbMmwFgmLwcKGBKHIRGSppWUsehKKSCZqOboAZfaqEmtuPppaoPWjTDTExbYrccbPTKQUjiJlbYjfxOwwKVAYdpsNnjyrCoxLTPZUiHUmjEQHGHaHHbzzpGmxybIqOLRWPDvvBnJzciBnOOnUDIyGcjgmQSscWgonPwyoFTVFcmeuLLDHbKIjWwKNWKtGFxryLRVhLqQTduCEakHfEsXAdppXMqoNYsLHsbdmsxPbDzuAnxqiUfSkAAzAYATiGGOotVFseeJAKbncrEBwpvWyZkTirPGGxaAqgEhRkHdWPWeMKhlSLnpKYycbsfajFCweeVErtuXYgxTwqsaUgQjwiPGHvuBRYImjGfaVeylSmePIUyfWSyRrIKGWExnfIfQkJuacTphCDAHlUTDULZQKTDnYcxfMksSEFiwekrhBfPqZmMiaEsZSldBxuObcTVCYEfETbijqKCAaQNxQowPBgPvgMaqduUvxxQQBQkDcYyJtlkdlEixWqoXpLCblRqabflcNijyJovzwJmdVuSHZxaIECdwkLtxqyYjaXgxrUnuuMtrObXlLXepyRrCIxukHqNbHJeagbqWjqjrPNvrcjCUoWxvTXDABZKoCFfrpdoKClHAXauTzHWDDtzdnmBOdwQfNtGmHwxAWAdxGuRLCErJFyImmtqLntikQhUdjFVnqKAMdhluzEsLkWwdDsveKbTirbKNlGlcxhHQfXSTLKPCaSmSblMMBVgNebOqZAydBxWhPooZXeacbOKReHAFpBaMVUzEnXfqxZMlEMSrdnDYdxleMvLEKaUDHCWRhkWKkdkiDBQdECIHWESrJTuePMCGvocfvCNZScMrjDcMrADyUPyHBoIaXvMcHShvMfDISEzwnwTvJsurpwakCGHErILJTJKijlBLxMYDiapRsgOjNEYegtsWzQxzkkHYcKFVPIrfgXCQQDevxyhUfbvMHjjBpriJYUWReWiGVuMqzjJBZaCAZdjYlrriCEdkDcgTKHeCLpGlcayRbxfvSecTtaMlniGfTQWMeiiEQzKkBLqLHmVydHqSUvGnnSOFMOXiwlhOINDYXbYiRpPuqXLCkTwQzPHItmsvmeAZIjGUyxhdxzvusgWUxLofarJTmcGTJaCbYmpLoBCZQUJgXqrynyMuILcsYVDZuunrrgdQDkJwIYEHiFlUIcZvzSIGHAGoejJfahAQpzkLPgKznBTlekdIPCxwCiKQCyaUIhpCyWSaLwdOHCaiTPDsxgQwjfUdxfVyDAZzVYBmalBJUwvFOUlAUchgvBppeZWjKwPIDDvBOXRhOoGLIJtoMsklrljexOddwisnUlWZAkLeEYSMftEelfBThhMoTYhlwTMyzPzgyaZCrbuLeJqgMCFQZUNwXYUeLOFPXKdESqhwwgxmAyxdgDUECsclsBwmhaFHHaUSjqhIxxlfhiHaeLRDjyfgoxLoLJjJxsuPKUseCqewkzvCgoNIBRuqjZXHnwyBZedQSIwCTOVVRwHntHkyWynHOHUJxmbkPJrDUHiYXQznWxoJZlLOCCWsmDaMjrLPBObZsZjDGsIYWOsLxaVjqpDxWTHAfYZMqAWSVYNQieSMtburqamtzDpIGpsGxZtKZFIRjnLeLbawZxtVsdjYeBoFGDGoXqaEFOjvKnDpdoxajTAeBgxDHneGIiEVOdcCbzHobWWxICjfEyiNpFYzJrPykdBYKhSbaDugSxtulBgTnuRJLAeqvKUIlKBPOSACUKpvFrtrbliBwbXwtAKCxNPbzqgIdXJYXCPiDszVtuPKQuQCGpjRoVvGHDdoQuVfigZBQkkNYMGKFYBKBfseJYAcABjtHGiYXMjavLbhEfbyhjjXWFzJKsLwGlyBgtOkwgeMdyBbpFolQnKdyntYyqIMkSpcxZUlIXAuLvCAkYKTAcKsRjHgZXScQewEwWiQKIodiOyWvMDdiFBWmdePHJPqoSnGruXcUeiQajpxiCYVDrhFROWGgepVOxTRrjOXobcTIiudCOiEVcLgxOhqSVNkGDjkMXSCWvoSXUIEXOFyLqKGpDpcyFpcujYZVJWVwWuomVCKmScBIAvNWnIFGMPUBfUdnMhXExVEYfzXCFlZRFSktDFpnoNIOAITQYYVsvwQhFmnZtFUdusRglBOWwEuCYABwXaTlzkHQllYBcyojsimsPZPraFMJfEmccwMTCBpaaiYJPHbkCSKISYmXDXhlmZQUpysaJiiSLfHAHSpZxUOVPpffAVqeAVbroGESppDthUGIJWmDwrnwOdEDihbNTipnIHuVkXvUiMxlOVKgrPFtlciEQwKEupMqPbmwjIBiGFtBmHKGOTxRLnVlDvQvKrrxVyVBFFzvDEtMDHbcTXVxBoJpRjCcSJJMMRuzfEsILtIEETDcGNLSbnoJHDTDDCCqlyFCcdksFfZPusTrsLZokSdBkmKOIXAVkUZgnhMIhyTorBykSBJIoVwbHTbUbciZVQRZzmTXqDgZUrOYJKvazGznicbAQAZdILyGxKBdzXdvTQPRvRetPxpGhYTlppJzPEJXWMRNmgGErPbCEeRqOFyqumJXaARTOjAugTsrofvFwyVPvGfgZDRHgvZUtCbtyWTLCHzdfWJpFsRbdgWSQLZAQRqHYrMDXasACHZLJJACnRMKSmGBdtxoJbwoyRULAkvKvpsqwAkLDNiexkIdaAgtBRXMRRNqGzPNEmVpPoNWPofERgIGBmpBHwZsZDmLdwLQFpCMbUoplhANFoisesQmPOFiBhkzsIwrtYFiKxqxiqNRGzmVrujJaHIFgMYYVEYADlAdhKMmoVGKwhPHxmLWAznwnHXAPDGDqxsSNFGkTRTlUsxjIaxZaiBqYMqQzUPXQvmpEIsdZJUAvZIxoftuBfpQWLlxulExSSYSfFyBuDrRqDGnbYTwwwffoDmFmaAmnpSvKpHHvDcLFwaodXzQXLaGWqlzDAQpmZlGyxiGQVUXAfkTCgajblIfdHALavZmQwQOavGDjahcgMYyeGkygFOrXuDCETnPsaWGQmwJwDGqCebyEWwnYesutnRYJHieZZKIJqfbArooiBkCKOyAbQJghYKInWmepsoBbHamNEwpnianAkWhXVhDTXXzLQeHfloWwBMNqbjjwPVLOHWaAHnoUGwgpkptqlwcSICldGZeHvaYeMxAjZoeIuevMesVhIZYTQUfQnpQfeNGYiRCmJxHMEEVlEyCufbkDAawKAwKhEBZWrQraCetpStKDCUPefgALUXIydeFWhZboBpREAFEXZiJWstnNLfIwcQyzJsNPKxuskFCTthIFFZrxOndcUvPzgMfkVSlNgdWxvtJxZNRLMmXBkPWTBlIpvUgVRFEOQWQjWYYlNmmmPyTboxQRJqOycFzQcxOSEfdXZswPCzqulbbCVMJHgAordUpOLoSRotnZPeskFkCaBkByGfqmZYjMrluTITDAJBYHMHSrgLoNkeaYZdikBnpbtLiMKppkPDBIHQrJRYSDHQhGPxnixWopgAWVEdcYOOHcHBJkKPrIFnyuSjyYPXmFXbOmXJXIInOuXyGEqPYhFGnWcvRhHcbNTxRwHwAJQzENjpaHPCwStUgeTlAwqYaamtMODfCAbNFcGPcWccPgXSbYGZCoMkAQOkveAkqARMxBYEPWNloMmklJmTBspILArthOqlSDspLbYYtPixJUrvuVnkEZzisUuFIYgMOqIhRAvaUfKwdGjgWtoQvWoqUEmRGJIinRiNevhuWYphzmTZLGrDjhmtADZjaernqRoMFopKsCATJHnRVORIAYyrdGVNXdzdiMlMnpAORdvoPMWOdYbkKvJWMEAkrxVTaEmWrwcGzUxoywUysiBCaPJOXCnqEMqUyWMrAYVPbmEohDHiUbUWBcwcyZleDAdmmhDTmCtjDnWFAHPlsUXrTpniqBtCLPnTezQTCnicgSBasvRilWwbRpQaWJLsVSiBDhlBrehEuIQiuLdwltBhGWfiVjmrjlicryfdBKXVitlJvOmqKSlremeKsmVFYWYxhGeRjdcGTRxwqBmaaDjRYsfcIApnpEoCKlXcuzTuWOgWGBUzQcrUoWZqSXWWIIWSiKIWnnFxiwqdtlTzVjGqLvkBwAMXIGkSEIrWKCmBZiLJIHCRGoybXEyYszRXemwiPOPtGcampbdVYMjUPeiPEKLUScCFpUMnPQeqYJRBYOoFlRqtjTicNskQqcIuAdzlYUUMOlYyDIaSsTpaTHsujWVSbyaDUXRdBgFxQFAJBfFdYvGJqJMwLlkZnFKrievXsYwGyBPIqWaEuxXsPiXtHABzNgBYmQgyOlEAiGLnnHNudmupskfzlocmWnNhgjtnPMMBwUmbSVszCupNDQeGqECehOYshGPyYCbEwvHpPAlAethUqkEUXudsjppdWxAFtdXdmFIrLcmznjgLGNflheupAWfRUFQAcjMvxaPSxHWzVnzVhpNooJdTqxFOuRgCcLFJhyoInpUNQPbFLKDcxnHPfRSYslnQeSqsGRabAQrgfVvOKUYjEyUQWsjjmoHAsEUNKJSConMdbjrnDJpRCZRKMobctHVjUdQgkINyhaiHbKrEtTiEjGDXWPvxxTmCgrsoVUilbMPAGDVqOpGSIEJaCMIwDgvLXAAjcLYIvwyqOvlzcONLJfthYvJBIMojbpNrHVPpNtWwJleYzfaZegsNWklPWZdFUmFtcwHjeiqsQrJwlHhghpgKSYaiXlumQxccXkKHZMmeSyApAnfVrtUOtyirMWIHWbhriBURTcJdVNKVpTTOtSihAVgQRvVPkzHckVSsrmfQNHUuAPgNNWMTdDHMRQptKuwzQPmvGVdZyFGalDpiedqVPkZczBnzTSFmJwKtsOorpznUfrXlIkAEzZqbhdbLqrDOLcVVcuRrVzKFSqlxVEvoSsjTihhwaMPoPKuMOFbmIApCWBPeLCaOfguNkbmxNptzLNXrHoJLFnXeAOBPoEFTTMhzbKzAPIABxKpkeVVUuHQXzKntABXbWerKxKOyKstAggdFplduNGHhPcujyNQecvbtQBsjsjQiYfSRfXahKjohiXTFRyYvLZDmUrKrQwDOWGkneGfHrEMWJrilZObDSgJDfJelAPdBnxvGokLdrTkQXkWiplMKsNMeuGcmiiHrmPzVYEQkQwlnHyFdzeNjtNYwyvjNsLalGEFzNXkzDbPbZwuQSIupydfixZuvnNPmDUsBuyxRIsqGslVYOhWECOqRKfLlgwFrHiclfdMXeEHTIsMqFHMdXBwYqvZYJMKvBNcFvSLfNnZTpHpUNHnLspmphymerkQKckCBjoRgMDLsjrmTDpXIDxRYHlaePEolfYrJyQyRyVAZqABFLoijPEVtAHzBeoVDffzlUJcfLbdJMKFlfSIWehXAvyLlaLexWUKmXJIjoEKOXrDGsNfIyWqJLCVVHfcFDJuckXSWoXWTthxEtXSfljleNFdhjWMeSqHsiXUBQBVuOqeWLHIsbboIeYIqskwPLLRFKTicggFxWvvBNYpTNQuEBtMsMxABAyXXKlpjXfgHZCypuZAYxfIUfPWZCfFJCCdqEpwHhNibhkSFUVRXJtKOdHZYGqnPePUcpdtCnNddfErcjAFnByaVaLgOOtVwBSuIPDwxvlnzWCRKdBpHoaMtiRYNhGTVorrlreoUUBELeocxvtoJSZUgWOFtATWOKkPmBazICMgTVTVbbMhxNDWoHsGDZPpRmaeTKAXDxUbNCroeoandydPVKCEnGMweldZsEvNSsQGBNfSKBjRcvnHjRRvybOVicLvkICeJnkgdvtZCfRfhkXMTuyJvjbEtoHBhYQsqrQqmhrgYwLxuEOVXfuAajEQsDFCMyRvtzAPsbshEwJVwffWEhhppCEikaRIMRvtsNQJgzAyoitTRwRqNnOnYKLmvskKOEZMLrjVwIxBBkCEdjLXdtdRFEBDoFSXyVIHzgyWJtQmkmHHHnqMMEtPAVdstfzmwcgONXDNtywFQTEnklrSHXzaRvNwmdUGKJTAZrFlXHjMtwWqusFAdkJoDuElZXqnkDATDScRSfvkIgBPElLDeiHQnLcUibzETdvvRDbcIiFzhBaUmCrYxNiVWnxvjBSXqSQyJglbFUAFgtApGPXKZYKCAyCOsantHBfdXLbPSlHIVuCEncDagboFXfjmkiCQAHNoTqPDmHSYAdyyyTvENTXNSIKEBwcOIMyJiLqAKofwzyfPBFcOVFilbtCztiycttqXUzeSrfUIJkvbaOkbGttAYwanjXzvoUuddvtKkRapGaZZySlscjthnxXFucEhCQQaBSVaMrCTNLZnwbmkPpbDNlFIfPiKDwnBunZjQvRrbHlZlkGXDFuDuNWwTbafWbAkxEdNobApjIkIVxcyPryUyaEHxKxuFUspmTrwFdwTorGdjWvhPXLzoUnjiOJJiBaUYFJDZOKSZbjkWYjwstFDuyTjTwgESUifMEmsHSakTvKgzOekftdpRFJQwHOENxDNtLtVRqXLuqrIVpNprDGYZSKhKWmTrEpYJTpzzkdzWbCNgPdFoZGLyuYVlcbKvFzdbKBDixyCThqvgFFAmZMghzjLsiwQHvjOUWvfIYYpmmYZJVrKxxudlcZrNZsvGDOTgJBUoKedJQSJEiYkJqCeycYVwgyXjuMzYftstuwxPzwlFHDYrIFQRtgseFyEyMpZguTIVCKZaJwjtrxoEcToloQYTmGVYYJVWPlQAnRpavgnIvIIxkXbLvAfUuOBZbCEZkWrzgWCdZXoLUNYxZreLRMfiLdJGpNeuKYYCBDFLhlYOtjuGcmRiaboadTdTooqIdBtgusulOsLOdICGecTqptQglWKJKlQfXSaevBdiITuIYZWJZpckHubniWAxhplNqBTzTOnCgnEABSIxFKgvTQUMMlvnjKTyFpQHGqeENphwyEuhhlMTLxxzemxPaZPNptaPeMGQLxEljwinINJNfrhUIkxluSzYWcQiTPJlJNnIREpjIHjGgVMBVmyoEXmzWmmZxCnEkWXQtscEsomuBAOIkPgjihWZYzijdChMEViaXMYFyqxCAddbYclaTYpLNrYnUakfsSEDjwQyaCJBOssiGlijEeetudUXzRLCjDVuVUkwuUALjpovgSzjCStJrmyaRiSctsNyzInnwRmgxiBjWXcKhvpmlIKUenBypadUIDTUxduxYafTvrQeYHgoXPsbRKzSOXBVesvGeGoDaiCffImMPiSinofvxyEcyYnZqKVUumFgrYJyZWfxyRacZnONbCCOBsNEZRtMsQgZiYHbuNxCzgPuDrdZqYSabKBYhBKcfMZbKrZEuEGCVMRNppCmorwqeeSFzHqjvabaeBYqamQXRCaqfPXhohXuJncIqPnrVYRnfcpjGSeosRpTEkxOjMTmpDXlaXnUzaRvypEMLcQEBuekPmDCqGvzoVySKhJcHllUwCbmeZLIdGCwYKqFhvPtxWPqIqzPLcQBuXczyRXrnIehAzPVmqzOQdStSjXMffGWSoVRaUwNGmFOSVTLfVafgLfJSuzCyRMverSneRsIWPyGQyZFwTVhqMuurJhocTHLwkljBLpmDYFNZcGSnYKRaeGvpkOPfnbgnjfRVZTArxUTHFfvAOFHSyLOyptqiNoSXuqXGWiutmmTuyIgSYvaaNxbeKVVkfZMpGcuPFFIHSbDwbKQBKqgEoTtYxUkXXRBbIlugCEdlaZnhtHcCZlgyUzBjzieZZhcmRrtmVXhgENiKYHsauPzWajkzYRZqrZIoeGIgWvYpkeFazMHBpvdnoZQApJBszPIRCzUmTQXdBvXwFhPDGRFffLhWiGfwUCnfLZLzsgQOXoUtdkJyiMOmLpLigUAfWjptwBSLEbkZMwTypsIMywoHSVucMeWmdUapQEZhKJumpepsENtkSEZwsmsVhCmbrGsNwKZQqBhChSvaFYgVpFDOhUJYdXGEpNoivrLIduFPiTCihKloKWAasalybHfcqfQXWvsNkBMfLwhHSlnfrmnvfAozIITQiSuTdsKHoGEUASYuqktbIlFCkDDNKobtctDOZSiFeXYhOottdOqjwnsVLUOcFdnRobLgKoOAnXbzWUUJaswLfIyCLgIWpiDpNnhontHIjWFlpnohjchoLhJInxRvTcafYWMcYntPfycNPNQBWeQTSkJdcvmhNtcpZbixwTaLnqNWEtDGkGtaxLPyIASyHJMhuBHrKGINDunNTwpeSoBJHpEbVRKpzjpHRALnRgaoZQoPRvjTsZdcfhCCfmhiRQAyQNeGdxNiaSoTYqsAXrdnCfhBTmOYGkCkTKYLAOvrJNkRrMNHLllRJEraoYaaNFvPlqXUVKfawERCDwrsexfSZtlBVKuFyuERatvRxtxPbZHzqVrWcVsKOWWiJbvROZcFWqbDsqRprzMvDHQeEbwsnCOHWLnhrxPSvpsVULaqlKQzKuMFYQctXCwQNdRoMqFTgtqoXMYcjWQpEumLXtMdztoVMAYwGgVXLmJoemdFhFEyOSLwRaqMSaCdJMtgMMCdNXlSALlYlIXYGnUZmHjchLIHWzksnSOlphPogTksmqXfBSksCvzsYktsqmZOvLBpwGULCQgztIzCnDILXoRkSgorvXfPaSkVknkNorrmDbBBeUoikQHmjOHIkaUByoyNqbPoEjaXIkDrTLccQlQawPZTCduwpNctpgOmSFCsjVToIUxdVnxwcjjdXNTUickbiTcnvMkPPaGfgCvAOMrhifXCrhzZnfMXnuQZKKNJHEqnLSQsbJPXsOqHASvTXrCxipLTGPecLDZAdtXLtAAIYWtlVnGlgIoVCwEvxkSXmQyNvdTBmKDHTdVemAjHtftkmCRGoEKSqXMbMzyesEKhZNmVhXoadkZATMAfirYjwfnsBNvXkYneAntBLWJkGstzYOyvbyUpuUvUWjjqfSyCiHzfbBGXWtqentwQkqfMAgJSSzBWNCVZUPepSnXMnMYQNqMGrnFkCZNfUpZwfrWzPfsKCtDNsSpRAgrgMKfKNEPDmEJbZWIUuZSfvPSOSiMtndWgCiiKFTFakeVhXjAGNGdCJggpywAXxHshHBPEzVjDrPseagjcJSKcgPMFVWflAUQraCBfrmdYuWefeDMytWPADftujOlugsCfpDCelPGpYPRbPNgrIpwBMnRJbGsVBFdgyTOKbLnJcMrnxFNHiIRklVOTAQEbRvQyDIDoppfLOcMzuknnrtQBfCagrgSMqauKZvjaUbaYyGjenyKeUinNsJEGwqqxikYPoimLtFWgahNggNCFteFlyOGUQzneHHZHmJaXCVUrskpRWVZbUoAWuxvhUuGuIkTRjHqsQsiRSuJiCqlTIPHBLWTokvNDLeBxevgPeXtTTVyMINYDcUjNaNcmzLPsEZzMpCzlMSRcVzOzOjqnadqQRokUHhEgOOuGLXgIVfYEYVchZnxmwpvhrrzoLhfBroYxnaynXVSzDIRRFTEdSNCjeICvrFnaDbajBmwmxeJRTqFjrAqOuPXfiyuVgHlnitKkJQlObNZdDhbCUpRCdipWyIQEPLUSXhtfdxbLnsraprIKfCqBulijAqejJSwkDgecDSZJBrtUOKmvifOumZBTmiWLRycjUthwnXVrVUjEPtqqdyNijjQpFIYxLRlBQHBQMNdrLENlJiDHvAUMavGfblxpHDqUMiabIegWdKSygWGofZzpqedbpuaTvYmdaQdMacHvPvruukJZTmKnMoRlSTQagoSMWvtmnCdZJHohkjBYyatWplDymJlCSIHQrgbqqQpJlSKlkzgYuxQlBfYMlriPmNPdFhylEuChlwYBMhYWcxFBTRicvtpVhEYzhyGEevgHGnStjKhipMRxbkTwzOssQPLxVdTCZJOdbTejCbKAQEumhjcxJWuafUFNedeJgeHIaBkPXvssuLBswQQzVCQpBoCJLxJMnTAAJhNFuGrgozceJmdCfTUelQjfUAIZIPCBHsSoFjbbYVgozTUpPvUFaVLIlgyuvZPJYMDuozEtujMMPjhbvcpKtAbCbANraPpcmPfBuDCOIYSuHUonBXRJqKxPvQhwdsAQrDnSxUDmhUAsMWPyZKOztShdevOZgkIRICZGoVhiaMEdcphLEwMBehrHFsxjqybQmlFLrgwsABsQkNTkJelwcupCggvmSJddIntPIXVVvwzzkCFQlbbLXnMsjTijxzKSiRNxhTNkcZGJtpFbaWMUGmxOVXjMTHtxoKLrMIpiGPsIwJHLVIMCTJYitcNkLCoCfZeBxmwaKXUIWcuqjaVQdCAlIlKkLmUqPtLisDSZqIEfxBtTOUFUUMtVGudyAUJsAoJQqqWAZIKLqgQCtOJaaUZqdqMvKQYkEgeFAyyPpzKkxMrSLiFZnqJMKhKufhJmuSCWnLzUYXobyhXeHPIZdZYJuIQiSjPpNDgngDgUIrVXlbKIfDjeraUkCDremBAGJKcjdNYIxjjoGbnzMINvZKmCpobdumxYfpsGYcxFipzmanZEEmsgYqdeQQghDtDLtAgEqlrTgPqWZdUHeEjZTVuFQHIchsbzrxTcZsAzJkxFWsJXkOQBXmzHvzFMCvaLcSfidnDwwGdaaQCeKrXFoadLMOjIjBKzJCOwdJnZAbNmWSrGiUVuWhaWDXKShutHuvGLrNTutgkopObamBrTXpHuDkEpVCgfimuRQYwOJjiYFKHGAZxaIUsypTiuHKSDTkoWkeIFkBkHirPqxcKaBJlBGAddjNbGHcvMYWjjwreKCtFKItfzUzKfhbgvEVIwIZnlSuompSfoCKLWBjUTUaDFDbCVkUIaHVKYauSocSJhQUCVmGkrlusYWUigFAbkUdRoMdViFWNYUEptXGIzHDrLfIIKdhpiGHfTfiAQCxJWDpzLxDmxBSGVSMsakgePHvgJcPGqeRExCSdmXgpdJFrYPqjCQfERGmrBRuUUDeFIQDnUxRCLZxtXQqFTCZJbpQRQHwuqpILtFjmadzshIRxAOjlvWXoiZJoNNMEJhrXQwnNmPtpseXeDGeJwvuFaZpplaiQiFZeRyzPVuTPcoklbinZhGftGQsOkASosVMZeknyiHyOdOybhmEvdgTMCMMCgZCZGdfuUNgNuGWxlhmcVnPvIuyuGXRvSmgCtSDHjRuNzcrxiUoYSQnsfXFyNduyGKguCuCFpcBpOdcDlynZAdCkKeLCtBTsFtENFrVRzrtQaoApreFklajDUTIvCgmzRrGoeyNtdHPwvCbnZzrbNUDOFrnOfZbHnZLEnbPHAsObmNgxLaPChVpUOUuGiWwlVrVUTLdZKVlxBWqaMumuHhdGOoLgnHuxileQOVFHqmwFRpiFIBFANtphPbjqzGkamBcPSzLAkAJCxmTQKFzDYmsmiLdJWxJCqTdleMycCBDjCvcPjFcgKxgRMVZjPLbFpEpyLkXqJjEZlBNmVUNTbNKnEbNhIntXMqaxuYslIYcIofWHSUkzKYjcjgkCPQhVMUUoflPmPYAPsnVbCbRGtpGyGwOHwTcNseiUJpgwYYGhAHuMEBKjJfUdgZElDXSBPXHEDPyEqzPzZNNuWksdTSttlZmXiAjaxQYFZKROYbrfaJezMlBXbxRQRJRZVQuycffiJQwEqkHulhufbaBWfitCSGSzaVZkEzhjDpCxVzsDYmSWneToxMutwPWVqEBhzgcoeMMmXopuTNLQelCrVlPldgGWIGMOikFkJtdJCfeWixbUbHTsNJpqTDEneboXoXjiDzbFwxNllUHgqlAucyyFesWADaZYVOKUGhWcHFkTBEthvzqXmRCcuyZizkldWHmLtriVmFRrRoannyxGewRggubkvawGLkxRVwOEeEVLrqkotywcJiuDVBPBobTAfFLIFCxmoupzkAIRIfNFmmArRTQDTaxbFjOEWGRyHXTjdZRWhrbrZGSWgxaCGQKkZKPHbAvpwXrsZNqaZohsNVIHqamNYBjoEdGSJweLbbkWquSRYTEnuMGNGuorvZqYsdcAaKPgmHJErTOywlRVYTHlpRFswJVUqsaQbkDfnQtQCuxxZdwAqWQMwHznGIVhBcDSwFtXCAxwIfTLPuZDXNjSstLcLCKGJsyUlmNgBENCQyUoLeBYcjirQUemJcPFqxnbRpNUeLrqtXKdtyiQqfCfUafwhdOGZpmclvxiKiamFSPpxOWuMUWtfNzPNCXucKwZKClWtoKkoKgzoKGTpaIXTfxyNmVMFTVxONizCheSXJOBPKYTfsgTIHJnacRWMvoiyVIKnZcXfzzEUVGugfxzWSFodHTIjHKIwqtXEbBcISDoTgYVPOPMfpqdVaZAiZRMODkwACyZmaMBpnQyKNehFcoAHFjrbPBxogKoIMBCZgxpHWJpyjBTOyCmIDGpWEFWeUAOsEVSsFJtIlaCOPEwUidJGwGhkbySKHxsnyuwmRXzQdUZHMInksmURAQMNOrzKvpJKfFDALBvFRASDVwOURyyADCVMRnqFjtGwChJCIGSZWHgdfoiTbsqFVAhSxUaSqgMoHDcrLBMJPtguqJvkMUhnttjzTZyakoTZwBOukMOFizPObRCLeVePEAbRtYPgKDmyfEIeXlhekJBPORCggjQrehCjGglvYntwEINnfzAXRrBepBoftPWkUfkzkTogEWcnZZjQdQDRsrKkrWJwZAozMvPtMrCtUYzidihTMyFpuXEgullyFdpquxrdrccfPwzNUDOPJVBweNLLdvYGfksQYajvuyHKPTEaUObxCVitFrXCWreeJicLMlsYccaTaTXTutDmNuuZkFviKAemqpXvCyBXjPZJuZZhBStgFVeLTmtrnWeHbHnpAmKuZCYcLaYXjeTTfLXdlMFHhuuzlLqeLhmJuNmbNtWJfGXJTgzbGSQymZDaggrlBHahgtzDjGxEHUSsSamTlTvhtAndxHfWEAZBpljUBqCrVvwyASwtICZfDbeMctbufpjtdAzVHaKhyfahLwHymxjtGeKRYbRzWUhPBEyxeBGrLcowpOQLcsNIliGSFIOEgLbwtWJgKOatBnGIoFOyFCkNXcjGVxUtntjHaWdYECSIqEjHPyMiOGQWsxXaqRhxngwxokqtxGsXUfJHLWfgQZelXcGMkOpKNnqchOkmVQZHrCIWojdWZUoVdaHerGhbMxUFXewddOZZmnZkpIxHUWFzMbxRbNEmUMZdoWJBbbGIJLlTxoEvHKwQbGZvyXqczOwpmJsdVBaDlupdlfcPoLnlIHXbLPfeEmjiZKeUwAXoKOqOQleYNsGIHbnqohNlLDJjiOGaNhqKqAJIiOCFNSHNnhBpSwvskVKZUFLawQAHdUQoTdwWUTAXKhNJbFWJGgbMJTtLqWxPfcMOxTgZwBTVIiOdfHOmtJvUpEAtZVukWTriyjvcpRviFNPLdiQZjAabpPXcjNDovwnnUDWydmbWJlrHELlnJocCTrIauxVbcjTpnGMUFsPDmXoVBTuPlEWsITAgHCizjcwncLrcrLntjEJnlpXjLobIPqCSpjVGSGxRupBIAvzrdqqsfYJhKYnOCsHbTzCfEeXzGwaypAZCUnNQMCUyktgpOzPcBHfrEwmxumpuzBtzlXCYfyrbjHvUPHFRmPXEYZnuHCSvLedKexnmSehKDZPAUtbCzSoDsoXXyyGMjgPZbgtBuiJwqHgycszgDYhZizXKWenQhUoAIIoAWfjhzraWwdaivGOmZgquKBjiXjifFOZeAYuuykzSGgNRLqHGpygZVPrMjMzqRIHdKkCsKDlMfGzwuIBLjYeVQmxVTYHoEjEyuxoNbhwqyANegyDCRBZUJFGEXnxfEHsfnWGqXrnoWuznReGVjjPalycyMqeDdiddZCyNOHgxiOLimRrxCsfbMoVSFhZbEwPilbgXLopqYMONMhwDOqfjfmAGJxiavtOCSnStHZMzBHmeXtlgiSiRUClWXBATaEDIdGBZfTUHSEHHnQthMQWrtWjwEjySXPOpKABPIwqIcMsfKlgXEcskDlUgrizJGagRFGHnUCzNLOctcGcKouZBuafAReknwcTfJtJNSETVTuvHItyDKSyKdjLMNnCnzsmzSQTDhtizdjNwJlmvFHMDfhEBBYHeaosxoFWldMQZQookwDRzJZIXIYwmoAGPXPDHMvIfHIKJPqRZGDcaGkBdOzyvrPXXUNljnblsLBJogxFpeOfspmySADYUaqIPRUHEoEhQMFUOHxRVNzAQRQqylFGRuySaKEHEkFjuygUaknicmxErquSGaMvnTCKjplPmCAqztdBEQcelyMZnOKqcAzOdYLJzRCLmsxrnVOXdIaHCkYWwLsnwCTENZqpoLksdJAshOosaKJkeRKHFnEcLiIrDvkbWpBWJYFXhhZywnwaWItiopnpmFBPQjhXCfpAEUZHRCpwpvBxnahajLQRkcFEAADQVquXSLiLhAcXusJpIDeRBZAKyzlQXGUCUdRPNVzWLUosVSKbhdGUlTHhnOpTqUqeASUPTPGNGSpbBsaAtiFVnpKliKNMlHLLTNyfEjjETLFsclvFclvUNLkXEnXqfLtzhUynHEUmVhScwcFmaXCTyFBlctUGONAjpomtjqhCGiWimFNibRNWIvCdgnAxsUsgrTQLKjoDEQspzAhFDOWSXwlVisMwTdKGFjFeGBPiTynDYcQcbRmzgTaXlqDwpRQQqvpkHEhxsbiZZRLsyGUHOqAPNYsfLoGqbqejwoNzmbptvJHALDPdwOtQfmbLSxeDwBuXBQcqFAzUkocrjRQeUXcPWppOQbImFriIJsDustoDsPPNAoHBwQWSTJpHhOTXenpBjiSZVXInmuOgzzZhJtxkuXxvfeIQnyBuhquEMBrMNfUyWEGqKOIFWhUQhUblWrhZihsDoUNZRvplPcESHoRIAJJKZlrAnRejKrALDLDMaTagiUdOWzNVPAQwJXeAAuplcdJUIHWpfTsmcoUKbNmtOOJnUOcRWGeBOEOAuYQeaDdFkbWUbIuQvnWUticoRjJFpvftANQhTaZectOPZecrDjiJCMxZLGIAxVeBcrQpXnXpDialIIODLESyFFApcSiFpuINGgmTjAxOLsZspaDKnLJRooFcZYzfjpGWAZPZEENhztDtbzUqCOiHZmMWqsoVhZjMpOIsGVymbyVvoKpLGJbDzBRyNzVSZgZXLdnmgIjxuQheyOPXfjtlLmxWoDPaCiUxgmBZiOIMCDkXoCZxperziiqdYPIPKMcqVSYLTxHfHZyOpsxEwqNOGkQmHAgXOhQfPTTTYqvDMHkbSfeQjQqUKFUGQvovXxuppuRDKanuuiEZttjkqwoVVYoEsQaklDmYOIuCaogINXHNwSaJDVMgGvnzbefYDPpdIrwmdbplSljpnqvVBqifVrxdYOlAIiMQHeuPzpWJPRJaciZOEvGHwDVOpvJumqaHWiCNWyVPyHRDMhfDHmSutfQdWVAwXqGnfeRlKYQmtmwCSbaYsKgVKlJjRJWuRPdFbNQwoZZaPaoGKgENHQGBhtKdeaTQoxxfERlvKAiZAfzRDJXrIZhmoIsKUDoIMwDRJjhyDHcqYJPtfNPcpDSJejwtCqvAOSdaEVgCwIFjzsmfwjIDcwMEdxyXbALkxvZSiIsbgBztquDXANkpQziIjInIsVUErmiJdHeQtrrkyhQhsKHzyxTHdxIQesCIgwoirqgKTvcMEmqEuROvEymZMVqPuATrDfUbKqnEXoaHCuiQnHVGSKhxxVULKMPzFCcruCEcwgtgjCwWkeHlfuPugcsRSdAGYEbprlSjRkaNuRKCLlZkcRIvXqYFHybKrxWgFtKxmFcxQARJYmEadbNcBnaszOitKdxwsBVYYppOMALfTkSwMlVyLCOncHDoETqcQstIMbecVFOIytPueytqdLwheQPedvHyDijJWHUABQBDOvGlkhVazPJGFaJUFKvtpInuPOOsxrFEBrlIhQqpeOQDvPiUWkJKDqOWsGonVtjeIinJDdkYpJCWzDdfYRjwuIUyUAcCHnUHFrkZanpxGjbbOrcNdNetXwQYCXWIpVxzPhscQrSPgNcAnKFXFuiKctUnWnqUNhojCNkrojKnVyKnjwwJSJXVygNzvlcJIFzjVmiyVOiVKCfvYHXWzYwiRKsAugIAKXkodKaeiOhNXBYuOIgKshFyGeZiJbsQmPRFCvaZHGMgoeYSiYnmixlsaWhXQyxlCgYVpOlkDWsvDUzXllFaKkevPYqwjqOViLcTrbcUskVvaMHfRZtUQFvqObUHOCMRkYhwhgHSNvAGsuksisWuEuEapEIuLwdsFoIXRBiJcXCeJTQSZnLDIpnjXwkfvMifMTxkHJsYXAmdRFYQqMQRwTKfRalmlPQismGNHiixFmyAgUsHLewaoSbMUAZafhfmMiueJqeGohMHmiKYjeEBCHNmyRJXZCaOLZwMXdsknyyqFNaMqqMFCRFELQjDtNDLyVVCAdCEZSFpcymBwSBPAzijwfbbEySlGqwScrnhOzSEMIeEqrZQOCtLWUqSSqwgOxWbUKeLCVNkqmCJMxOqETbepHVYJQimgUlMZaCmOqHkBaHgCulvpAOLVqowdSKRZCgRTpOMFGVlmosooQmIHLLpbAAsmQtlMXcLGTPdivkgMYmHrOIOPXkctUkErEFujBzEfkEgJnesqFfMEqUGJJBIqrudEXYbMVZayZQILrOLoONLvcIIffUBQcNcshlNuIVNgnOizkScDYlJJLQQgxPkcFqKZnzxMlnHHCMwuwjynqISTGOJGXqxngKCvgSbraeqeUkvzgOQHaHqcCPpkybxIFJSyQCsfpkEvWDHpsDgBMmqEmKDijOBTzyjSnAbWDZDpCaatXrJRKnAyBwlrpTQvTozCtYuzTIMGGHzFhQDCsCTAfRgcOoIcjvQzXNsvDZChqCTNUcoMMaGcTwADDfbJYpkvjwgolELeMqODzbLZYEhEwwzbONYxRzVrMyAZsvzIMltxnvrEJTOxYXWVOWvUjxZYZGlxLIuugKzwiyearLLKqDbUvWNkZQnOHAtLnReocDUiuFDTXzYcptKQhURJonRuNKXERekfczwXsvhhpeYXtaHvythoVQBDKHYjoYGZMSYViKqAixJsJMHPbFctKrYXVnKPDKUtsRlkngeIXXfuiCxoTmKtpcFjAdfRriQxDeEMpZgKmjxdYbkfOzJsDoYSJrCJnvoneSsECdXjRHTnXTgmNLwnTJJEnQBtWFVsifDDxTbZkeOdrkwnXwqKIFPZtnkQdknZxiKbjzxrlpbDAQGjWLgkUmEbgzXNyJAeevsImdAyTDUVzrhMZRphWtfIukeLoqqhZzkWGUuZHpUDtOuzsfjClKebVDxCbqOMjaTPUdvaOzqonQrjhNMAdbxfAIbuPUJLESehLexMSATHjYDUkVgCliiepsuAbLjsXigZhFnZolVIxXqLYNybFZheCCVvmsCFIAiOYHPexQlMMAjgCqvTjgeobVZTbVhFsCjzQchGMkyqmEhjIYdfXrqXwhOmyIYobdUheQrExQwEAisPEkecPsyDRLPHxpmZLbTTAOvKNiPSpuTEpvKHMceHpoETifGjthigbqrTnKmBthbjkIpjcKEfhQNhhsuAIaBKUrngVuVderVrlOvrLWKUycKwUhgnhqbCUocvkgvYYwcBQoicVJaTsjRrpYvUHSHrzlQehBuoLIOaXvIkmVcplPipzBEQDEQVcbZYcgLkSthWAIMThRYaAgHfrZCVFDzgpKJzzYQzjpNRCoBrpbsbAjSwNkKfBHQGMuneBRGlQesXeOAXGzEtDKhBGerntoRDErsWEHyPqPXuZUPDCXGrsFmgYtuHzHciQKjlQMtEgMXWpHfrvmPJDgCZpHdYoVvKNvLWQQLWNhprXoQnjsNGhQidijiLGnOFqaXLRUGeSGWVLkJRTmszDhErhkevcFHuzdWTCXIvNNnKzbXkuvEHutDTccdAqkWsZBOZoQFdnlhzjrIHqjPqLeJZLdBfiKpmEWrGcoLoNejHztDWrMibfKZkdwePrBIPUFRlvFZdbHFTUcnwKKaLVmjPiRtDIcwplBdRYyswFVCNtxvIesHuRpSMKmQLYnQuKGYQbdecmEfLYEuPMGKfGtayZrIdFmhXIZLAOPtfoofsMIrGkCFDZMzNvMgZBwRFWKpMuzueEWIjGGFMQgQGWagqEyMipuzPqoGuYYBTbeIKtquaBpIaPDBhHySyLbKcJKsMsKBVQhVriRqRYMdwiRoUNWsLRGZNCqyaCdzheMhmRyscNZahSumwRZOBQSTZUDtYogQUSZyFQOppabgXMRPsORovKDaNjaATVsTwGkNEcRHxhDqOsVMKDKfrLEtQsKijRGrfTLUgDvShrOIhMVpBMsonPLrqVLRYyfMzSqIikWZtsiaLjaBpetclZRpmJioToTShMaomNCAedcYKsmqwntmrFtopJBgiDUJAjinWWTefagnWJEWOSYyMfoMtfvzOnnoSsbekZHwEiiOaTSAPRQRnMRdpLyNGJNwbJNjfbtyFZOjCrcPxExnmulQcUspfVUcPABXlzUzzveEBdRrwBjjqNLwrcDTayHTGeQjxTOaVnTCeqVBrXPPrmUfLwTZVtqrSXQfYlWbIQKFZJaFgYAKgtigmWQabWVSmYMrbvGUXoaQxnJfrHkQavSYojIXoOqUHjZRyQQmNwgGtvEgLxsUywAQPxpRxhVZwzYyGDkFnfJdxdNIvhkHqDRCGjUuzHFLBeFZZDRejLdCmyVZEUFjyWHRmQBehtZghgbkklKIuKTgIQmSxJXvczIFgKgdnjagAPMCfCMZWlLJRdSYSNGygDSoHjJECcawrGHgDyaQndVimfQpAJzXxzadltFvZzYwrmSzKoNAmJHdzLYpXPMITVMTTNLmKIWzJEHRoyXjhtwAnQXABQtHZQKDCPGGTwFyEGiqxDMMZeGOOkbXCtbVVJyBpGEQysxLXSqBcIRlWAEDkesVgDzaaFtDUmPahsQvkERceUcKJqMOCspLWhYxZcDzxFsQlfXOBwYyozjrEaChMqZLJlLuwjrUQnDGSatHBdouIcAZwSTkdisAbQtZbUrNzleSVyldsjrQoGDjVcjBQyhyVdjxxjAlJimpOGssKFcwiWGSAPkQFUIyLCHnpOhKENikRqyBXKPvvzrsfHzmVxqHYyGMvldTlrtIgIzKYguDWweOVlthRIMSeRWhZVRKNGiydfLSqsXasHaayDwUltKRSfoJuyIgoCzmXsowXeOqalocegGxcrJgmcCREaedMdoDcJBrwZhSrSJDstwkDZKkarlkqrAjpwEZJxUZnrWxVHXWcLyLnnnTYmdlJKFOGTJjqWyyggfuAYabWRroiwTUQdskJmZAoqXxSLVMqUgAaTVmPgEglFKoLzzmMLZOhSFmiQagnrMGGqVtiRKBJOfRlkffPtvsLAAhnQkDxIQGaRNQvVrKPicYECVLEOBMunoWHEkxIEqwrTUXSqcGkWVRRuFQRNFTgFtsozOhGlpfxfmkOoEmAbjzZaGfDyYHxJZtIJPpkeSSuvMTquHOhfTaotzAvrRcRaxYnrxgkXIckBXdcVhdiatLgHuTzCzZuFlmjbvCFTDwICNrWhNrzfBekzqKgkGAZfflHyCePEkudRgFRzcYSFzpbYJNlkDcKnyPSlARTpmXHXGVGSkOSTWXGvblMSFFtdOUeMDEgtylHnpCmbvEVgZLOlRPdPufnGpFqDoXmkohXSfDPNjZcahcrhnIzsLRaEPFjtOcrHdpBCTkKlEmnfkOFbPxzTZjYDrqQaINhgaYCmzHJijcSPHNTQzVVOyoAdWOOdhpTNVNQrxPMcvCdrXXvjIUfgcxoqFGJyjbzWoclSZKXuriRIdxIuhwlOPRDnbHdDdrBOYfskvRnsbPSiFlLMyIVfYdolsWSSBNOeHKOIIFNClAXzBhQwmYmiBORGYgUrwSHsVHRslvfBOwGeAtfvhKQKKDxikZERINwmbYBLxRQPUyuGerkRoqGCgQQiIAEWRkGYDpltGSxGsPdGcLHPgNtPgSVdgEIfJeWrGbgUVSzqHRdQVWaqIyaUismyfAOfHjCTUDQsSLxOZWWapSuQwKzYsASuKgKVgLjoNGbauyrHIWSlpGzSEgPNTGvVqQyzsDVrYOfkbXFulKRzMkYwqmGapSLnXkzdNRRxlfpNPmyrPRTFQoDetIuxwkOuMazOVCTNHdiJrzEBMIvffvkxJohlKRKXgcAgdsWxcXcjRfusKDrEYQJJTyXaBpEtirJryniISWJgFaFHlAEXQNDXtHSOGjijqIymkCmFzJukXIjMgVZsDfYOohFaLvKuzPiBqsWWeKGmBIDeOClbqmndNPjPZzsqXqGEjwKjmbcxNyOIZYIcDHbXyxdpJjsWRgNIJnznRNlZuLoZaDFsPeoQStTivpewNAwfWSykwPDVyrdVCwmxcsvEGvvADLxEVgFsRIlWcDCUiMBbRYkmJzRhyaFtKfggZFNDTlLEUGQaJqgyOxGxxxEffcBarpojpNdiOLVoppWJHVoZjsPGgJhicZPrWsGzkpATbwwikYptqJiZWMwWklmpLtiXjvOPbOpFgRcdbBuScweWxJWKDJYJoIFPMNXpKesEHJvMJUEOwOPlBUEnyAYOqHgLjmYEebPOwlkNmlJycbOFXbKYiaWnVJtBnjmhbUajEFesrntSAVuCpbddjEnCrtnNrhQxGXCZPsoISSlViTempEIBPsdMBelmmUbFOeaOUEKpgINEbBeHeAlRBJauEdsVVddBCYBqBwBmeIeWopunQUQNtISpKyhGmtiLyDaNieEUGIpqFiwetWsDBTOaADNuwZvWfYShKDuBpvRdwexghGuWHsMSLahAOwjKePcmlKdUMnFVhlanpGXwivoIHmuSYreNvMZdHGFXapOecuFNtLYaTUnrSrGWyPpKpfkbQMilZYYFiibqWVmZqQdnUAbaSKabzCURshlUCnuHjxdOWqTewFLOkcmUDPtbAgyWCeinNtOuDdpMDwMIAPiXItfWcSTRyDxzwUZQCnVWCkFQzbgZStaNzVyMLqDVCqpDHkxkbceodZVoipILIzoVrBedbcIqLHfJNKLdBSmhCRZVgJGTkKgbOOfPArpcpnXhUlcTDsnYTgkHFYFeswQDINGZuMigewgKEzisBkZOFlJPAcvXmmbiKRVmKTsBEBKnlgvxbhWwGdwdzKxSQVibSmwcOoShNBIiwBnNRCJQpjuFCLuBfhTTcFOAfQAcHMfbPektosoHFkgSiGbIYXBRmpyYQwwGBoVjSnHkyjWFytNCTwAYoHNJFWYaOPgvWsZwNBykxPSceeILhlhGQWymkVBmfWkDKJWfrCKoyUesqINTKNpXrMsNLtCzrSpJTaeSQLqxnVbqTWoxqUcLHSeWLWgMxopEQRlNPSvJSzFAejgEPqLPydqpTafeVZwefajDunwBxnhAvHFSjdtCZAWvWqiEWUDLLfkqMlDwarlsBTeVvqfSfLIkkjYzweAxLpjFvPLYSGgIpmIpHkaWQMKBGFsqDEntGudbtMofdfmmfbRUORUeeWJvjLldEEvblmxzRQArGNlVlUMOwmnqgLGgSlpnFPippqMFAQjyZdTotNYDZxAVBeFKyjDkYJPfSOzSThppYdwLFfBmsnCOOKDZioxGprOiikrWeGsrKFJYBoWcumtcTYtzJtyczzsYVTYrLCFJbyIcMmsLHhmbbVSGbDyKkczHamMOVToaCYzjBArnXTDwBTRmOIrIlrKrsnZOafKEcRLFsFdVKmiUqMPaaafvpuoJcXmFpSSlbdmQofgxPKaMmLNiCQHJeMlrylIaRwbeDWxevVGlSfFdAEUmodeiwPYKEnqmCBlFklorURhPXLrazmgKGXPHizpFmATeCZpfmPIrVAhYpUjwkhmzBSwhOBwSdZdxBHFvUZsmPFbIqpZMfPWsyAbPKUUnfRRAeyRoxOVQoiAQMftzyFMWucqKywEQzdulUiaOsXmdBhckxdKovdeqDpnLOIfRaRLQZpQelIWaQsMdIwMnRzMLXBhSVeTYrFnfyRtNgyVmmMsKMKwCYhqCtGrgnXMOTwgPLcdDrZhsqIbBMUcjkncjwjwQuDiRGoDtXwdDVYainXMluJdGsfKMxGUJkaZzKQwGnSUCNqkqUWLOfXAyfGCQJAYdfvXpFJnyHQJehwfwHdbFnYSaPlTlxPuxEsObrtFhtSfuyaYnmedriYFGwizyFKdoXReTEawNjgXBdtOTlOYDVEsqKNamgMaHjNnRcJBLeIGXHBuSAhvExNmTgbnVGIxYhAiJOsvKqFqjujppkCsJYUbADArujmKLdjumAMhVEdcuEYBHWdMZrSYeBIKAmwzeAGCPfpdnGHTXhMxesHQWiEPzVhHEndHIjhApYgfOBbgXukxGqJxNZuSjeLfcoiNvCUdiHjhalSvDecDhVCGegRywXuttDcPPpmgqxNYaWkaKUzhCzYnZZPwEhKBvKRxZevGdmvJqdyuqaAQXchdBAdqerzDwzoFTUaSxLfQbROIuXRBBDSrnzJHqvKGQpTuPwcqnebtRgdbfniiPSZjrJgsppymacNRxaEDyaxlBNJoXnmdVNdXcdwJxjofGTUYBYyOONWYxxrOJpzslCANkUNzuLtEnINTWnYbAVDbjWWsaoQrYGFtlrJOtXhiWfdYSMcAcZcjtbxghEydwFjwdogKqnJjlgginUPULMBPuHyxFockfPJoyeiXPRONfZHielvkwIlSuvNOvIcYiNUWPIBwyCgsWhMtlukUpLXpsxHyRHLystvoIbIrgZoFGfRzUXFJmXzaCvdtGZJbqHPhDodJQnQGijdTlTDgLTdNluztLMQjNkqBwhaVwGyUtJBIHVLKarGqlmCboQfbgJmSllXRenMMsdLOziBbyOtDMIaZQocvaCMxNEkyUALXMzSnvlCbwaphXdIuxWmevyvEqHdrwFxLulPoiUbJHJlWwZqiRKsuHkLDesagSdmxtHKbBKrgmbKtxJPwrJWutMgLJXzDBObGTbypBIvElBHCTeDjldAGzyqtIxjvVObzNJjARgEtIsHgNldeGmaBQEnbnvNSrTrXSlCCmnQTvrcroMhZLhuFkVNTmRRcyqUlxrSeUGMgVsCyXmGrfBRFbnCRavcrjvnQALWvMbSflfazFuZYQBvBcJcBaHJgZsQTRsLnDCprvpmNcanjUcsRXSbFmBYguiZjNOCcrmCXInbcIkpwBLEMGwnFcSQZXYUwUMGQWYuTQzThalYPzAznnMqjnnhUdAyqVsXKrXFGGYcFObFLiCFRCftqNiAjlvxkGkJnIYCHaqMzEGMlbLjzQdndpDtFiiLiaBAVkVKoYBrBFfDLMOoiNcqWTreMMcglcjkFXMEqqQNcoQJTIeuYluNFnkGMYhfnRkCBNvStmGUHyHuelPuZBMGGgIwFMXqjXbkHYEExPkYFVLtxWODiEPQxvKuXmcVHnzOmXQrlqTJPwJFyrOJJYiuNNFPfIqikkKXIetLAAnNInwPZeGDfippZbXSXrKYBHRlhzAgQflUfiDwdqasyUOFcrDlxKgyKXaFaySZbyXGRKiUwuzuOlXpDbmDHXPZAdkqCzulEeNWOlLWTbVbheZufTlShQiuSzZTKzGHaMzHVgCyGTcYwYTxzcNMXSuwvTvZTmvcLtgGdNBMYVUBgWeigxgtoYhAbfeMbZgQJdWphlEFjxTKDYGNXpXgQPkMCbuzfzyuCzwFFXlXUbueQrnHUTtbDGXHXMZ</t>
   </si>
   <si>
     <t>2026-08-31</t>
   </si>
   <si>
-    <t>23:25:30</t>
-  </si>
-  <si>
-    <t>2026-08-31 23:25:37</t>
+    <t>23:42:23</t>
+  </si>
+  <si>
+    <t>2026-08-31 23:42:30</t>
   </si>
   <si>
     <t>{"key":"value7"}</t>
@@ -668,52 +647,49 @@
     <t>&lt;root&gt;&lt;key&gt;value7&lt;/key&gt;&lt;/root&gt;</t>
   </si>
   <si>
-    <t>9223372036854775799</t>
-  </si>
-  <si>
-    <t>DS</t>
-  </si>
-  <si>
-    <t>kv</t>
-  </si>
-  <si>
-    <t>hJ</t>
-  </si>
-  <si>
-    <t>Hj</t>
-  </si>
-  <si>
-    <t>fnyIWDbyYiEGlLMWWUOsmbPZodqVaoHnkIrSOVSAUsectttCnUQfyDjHaXZqAGmnQLzlvCHpEPEFuOLLKTZGIGRMXHdvpDjJkmIduSOhbpBXeUlSkQONYJIsquDoavFZGZLZYUdahUshCbkUfdLSkiMLtXyHRStMEPJmlFndKCteFlVSjttXvXzoaqqRUlaVKLfpmZBuDQUhUaSBmIOvkTERukhxvFqzybWpSArzkQXmhuixxEmBWV</t>
-  </si>
-  <si>
-    <t>TkJtqFrScuSMyMTyIYTWWWyofYASytXsQLHASUyffEGDLnhRqydjJCcRRmLScziNHwKVDkdKuWhxTmkZsbhLCcGIKSDNKVICGDEHjAIRtiRODmhUOGZtreOhlLHPprKPTGSkGkbSUBBwjiYdN</t>
-  </si>
-  <si>
-    <t>zygPakXWSLTPLpmDnZugnbZKDhrVVYCvsLhaYCUnbhUmmEyRKnRPzrRBGzTKpSsEIHgAiabxfFLlYzf</t>
-  </si>
-  <si>
-    <t>ibIyeZsXKQhEWtYwhMEQwwWzBSScPMCJtVKQkmJPVEEbJFVuDMASqsCifEKYZwQZNBXSNSrsWZByFMgJzZUidDBjrLyyCAnplukZzFocjMrSjjXvZqolBBLISmfhQXhBi</t>
-  </si>
-  <si>
-    <t>ZdIskyxQxNGkIJMOkPXLeyWyKUfVmvcphaGzXXEiXtpmcUNVXaitanSGARORyfZlGsjrRIOJTrvglnNxXiStaypUtUVKnOGMfNgLWkykQEZmmNZwhXWqPHRWxfYxibjFpCGdsVhiiklHzvzGpaqsHAHUTnubZypUGcGRUFGQrVeWSCwRLJQfGvcaUhYmvWCBhZuDXoJNtMudRvaQgBafJUqcbSqhxCledPyRrthjxJznUUWbvQhrrGgwKiMokVlwoTZYmamDUOPaeNIimztxZUCdaynipQRFoXLBhGlRZqYkkYBtBoindmnObptNpirrOaXTOnuumphAzpdQVDurSVVUUFhevYmjoNMsfIVaYzRbWfpnlRSZpINbVlWSdRHEnlCWzmCLlyFQvKVFkaTgjSZuHfLzWSBqSPmLnbeqBThQqJrJOlosEktbPktxkQwfrSJoFYEkyaZqrCEynZFdQODEjFHbtRkDXKLDNCMwyRMtNAXBmxirvUQTfwDKtOIJXtcUzRVDoWfkAGmgsOGpTaUNuEpPfgaIaUadQAbehDqTrAAVgtGDqhZOpzINxZJItzQRxbthNRCVVUJZhSFrSwYHbBFiFiVKLiLyBBSYXXWzTFhvqtLclbqmwVNnLUwwEbfJkCEmXrcPOjZxMEnwByxGxeHOgeDFlYNSatSnElsgclNrsyXNKgPskSRoZXLIhpUSvTCrUAJutjbLIZLFropsAobAyFBbuHibJncFkECHWuIyPRAeafvxTWdmzasZlryDeWMBzEJLynKcepyWIFayrEcudaVBBdGYAhLxGEHjHKWvXifLEpTQlzwKeIlLGNXYppyqJWKugyLqqNUHPLXuJfCPbEQkJytuEjMQKZqgTBpeEtHDGbJaPxfDdNPXwsGCkkLQCRYKhJZRQBTBUcFxUywYDwcSXfYaHzmjeApUsPnDxKoHAYbAmnwmogKpRafXyRSqjnouMzviQKQApERjqivYmOWSANFNdQjtCMviQaIhrGDIsKUoHlDbzYkMtjCukZeKjZrejjkcCcfEurZmVnQcnUnluVchAyeWJxACOoNRrMcsyQDyXaSfEjWXmFLkVXZkMHpbJUEHTMTAecVqVhJZmCwkRdaKGKqKZbkUFzkwdqjETDAYDWoJNlRoKVpOivSOtiEohpneNBrmlldMHUYwAHkrzMzkGcrfjixwWmUqYmOoPoJvxXKvyjFtUQsLZkilrvaUyIzHEDbXCpdjKwoyPpcAEKeWZCLolusfnfvYegJmkIYobJmWGSViuTmKnAITctxDEBetxYkzcMbfxPbDMsfuUeMOYHTluYHmrnyLWbeVFKnGTJZAsQgDFNJCgTlIipYjyBaQkbvileVaOevigKREJRzEQJBqRvZcqACfewIjCOSFFjiLVRVwWqjnIpUPbHdNACDbezgmovQmzXdVHhTjXyLwLajJKLEQiNOzVBsLiWdcghRgZkGXWdKXfsTNdoFHzJnDJIaOMlHCrvyqSZLJEfJJQseWnuBQICYLZdyHWlTYslqYsDDihsxYUdIKRFxqvhszxekvxBzHtfClXQqkMXAvzjVfrroXqJDruiveGXSOYfINTKMBabdnmiHyXzEiaXErDHFdbxRBBtXjBgWYPrjKaAxWtDiioBmFqjhDDxYFFuMfDbflZeVABJGwvhhxPdrqWJIonmLNLGfQUTgUuCOsMDvSWiPSzGOBZGEzWNUgZGqOPlmKvLcWTPHxPPwcnUVCYhsHXdGAJoEVKLkBJceBbBVQIqXFFBVBwkLICBxcRCPSJdKOTUfFPwfTWWARyPAuotXFurTmxJAxhDPDgtlLArsKMPJVrUhXrpawTFaPyzzIPNFkmiKQzeOKmpseixoPDtFFAJgltukZvpDeJOZiWkNUwOZvkkOPMkEJvwqoOQBPpvXdXMeXFGyRliNXCHeiSxYQjbxHruaGGqQhjOngQhiHVxEvygJaCbuhmaajudzevGYjaWGaJIkwMpOdpIYlsaEwlJbHIZBqYGwTVgVoomsqpFyIOAcveEMuwvVROdEOPNGYtMLEULZjdaJbcFxKXRHKNvQUHvRdigrVYaupihGXVRQDQZUZfFvGJPRwQCPrKsChYWYpmQZfmZNbCSpaDdbafENLCYoAWYlrouNjaabjYHdoJmuIqmBJtxdURDEohJIiezqeSSnxUuJJcZsqqeXnaeVoNHHzHyggvfVmpFlSkTijRhSvQqPlxIyEXkWiniXxXhvbtwWomQDcZpvHsUwVcejEZUWJmfIliSYYYENydoTSXCIFozvuMXnTHZXgfFToDBegAkKFgwiVjtDyWlNmMmHXYqDFPKBdUbqVTJUqCBrhTUOUNJrGbvbwEFhrYVUYIpgvhZErsQXXaTMsJEjGIXlYKwFbdFpAlRbclhZkcwFHPiisVOwtEyflnLdTIELHTIRXVZBBOPeCmeWeguVJUCxoPIIrNkBmboogflDEvwfrLkaItZvsrxKMrXYJwTSbPESQXWsJnaETRCpxzCMNXgBvMCXpSxXRqdvKMkxBOYOqrPcNKSBSgwcpzsIEmvTpXvmgvOLIQVzpmgUyhkZksNkeQxuzzBPWeqMcMeJrRDazStivPUtElMUlXjSLHCgukhPnFRjMNwIjyYXFTreYmdDfJQluffByNuoxxWCTQXoDvhwBqIeuSJFrbTlVygEPXwYRWWrxymCkmIbLNTNxGxklsCqmyzuBxTKKHSiRtPXEddypPXQfRbjHTjHZJripCsXqQZJsIUkQswcjNiUuUsDLXfClUQZYpFhFurgkRaPiusFqPlBjhccFEUYHwkXkwkWZRLTGOTnPAmbUcTihTKDUDxTeEvhEQOQirSoBuwtqnnFWRTVPRCZssXBRdYTKrertdDaZoXpuFNZeMIBevTxQCqExyjtGhgjzmHcmJVvmJLsxIxyvLRkgvVaqDCeEnuAhSHWGZimHEQWSAWXvOBvaWbQQUiwwLvmyjOPrDdDEofLlHQfiGoJOZZeXpJdvRLRZoFNmSpCTtokjKuiqoNioQmCsOJgWHhOynpQFWDglcTuzjExMCVhcLzZCJutFmAKErhCZqcBHHFritXjDaYTRlmrgZeSzYysReltXVTASsXiVBTDmLzrabFmxYPwIcxjheuUBzzPRUsyIbmYPkQiVpTBBUBKcneIYJhlVSxYMoAjnhwSxXHlLsuApQhtKarJpONyUSkTuIQfIkxvryjiWcIDUnXdHnxVNzcOTlQqSvUyCwxZkbPffPXaemIRGChKtBiBBAzZDZAmmKprlxnLfqUutFYiQKpcqSUJgFpzENeRzloDvIpcsNckTqYGOsEmYLEIiqbZdEokODXBHuqbXeVMALZePSDvQvyGeeaFyCeHQfwlhpGzuSpTEiNpTUOAHShLxOBjDAhXymvuszWhOGDLqYvUSKOeOoJTsihyLOfoibmsZuvuGwaRSsrqMGJRzseDbCrGktXGEWFWqiMzYUFTQkkYupAwOaZBUvhnmyTszpUpNDZioilDkgDXjHhBIYYNIvmwtOhGJyBVkfDtOdcBCyIPWQKidAHHJrnFfXusGBQbqaePrcTuHfTzLHXDhxyCDjYPwWOvCogBLDhXcQXxNyiegMgLiBcKyuIVXTKIUJdUtqpBoRJPifAhbSCnoVvpabwKIomTLGauRtjWobrXXyDThjMDexSoOavdFmFoDaighSXalpWRzhGIUmBRGDkATlCxEIoKMZkKatlScICUyxzMJKpuCnveFNdSRpZvkiQSvEuJmvRMcbQzbUsPvPYKIDuilRzkOsgGpVSxWdevkQJNEwQnCyOuxMcAlVEhGFWVGPwZBvnZSVqWQEEiySMMUgspitGrAUmcBWvgDvSKmfJlsUVYKLwiPdbBgXRAKlgbeFjenjYEBMndQIQuXntDxTXSQjMyXsbBaTZPywbayiOwZkfvaLDIIIyvatjySMFSBdHTriRPtubHsqVwUGWZwWJJFQvhvfZxBUoBhbWnZxcnDSgzhkFSGuzIBYMafsrgTzEApKrqNfpDmjGavPodqufSEYKbudADDDOJtylzLtCfhnyLStzaogbnXgiJCrxhDlZhkQwEMZcNJfnZQBwAOhmzzmYZKfdiwgSBrVpLFoxfwNTlVNFIGMaDWHCpaZoDvalZTlFDLykqWZeywUhiPWlGclpVyEIwovMQhVOBHoMFGifvYzDYQoyktthrUDBADdGAWUXhICBZdQWsHMvTOwQbPfzONKcLgtaFwTMTWEagRXrIZzOUWztWUJdoakSRrnzOoMisQUaaoGyVHHIVZignLQMdoEwuWVPPTlkubwbcDGPUYIiPCyKSIeyGnnikMsglTUbhSgWITNjRmemEWbRkpZZFUaIvWdVdzWxhXiPwuEUOvEJQwusdBlsZJzPSfwJxkwjvLvWBMVSgjDDdhkpmGMrnGHukKqrnNVVTUsVrPcxyKsOWrFoAHNtmMGFLTnAToclpLAphAnGViIlCvXNPDJejJCSMElbpbOZlPraVcRtOJFbQyubiTOPEcrOAPODIBoLhEdZYWxqLHpgUZqYtQWaDNtFdGYCnNglPARaTXixTJJsDmNIAhlxhkVxqanxQYsVVDyBjQsGwUjApBeFQRNqltkwPzVmEXabQWOfkSssTpOqLkQGoeaHIGJZOpZnjiMUxNAxfSRczwZNbhiTHgQBRRnRAsBmRlrMmADUjvsjPtiqaEntSzrAqgNzxHfFZvnBZSWqvASdFxCgotESlhYcnHmEVbgPiZvwUkXxwNZHWEOryCtArPwYqKbSDHhwqsrPeNOQEMqTvNNdSwRHgadHcDwxuIfxofgbBeLaSaZITBCnCHhPPPMcRSTgrpNjETMmcbkEevGUpDqfVHeySwWuodOsIPwghRlzBFishIUWmNshxmHMedoWlYLunxtntGKaWoZZEFhJTxXcoONyHjnAbIsvvQVaHMXSRMyeOuxpZprTaZuzezGZoKSQwOZdDeVArKpvUbTWCsEwANCHMFSjvAuuJMXzwhoowjNdQocyhymuUNcACnNGDYffSeiIjLRQmqTPzosUHLFwJQMAMWtgIoEWiYOpMJGHPEPqYEXPHhvYcOYntGUyOBtwGhzMvXCKCuHcbASRDaChAfQacxJoSUaPZCMCcjthyhQgihfcUjDLtvYmDfMoTxubXCVmqHfPWWoVXraYIBkyzYsbZCDVBSuoGfaNUKLdRPjLuCdlKtUqmhBoZooVCrmGfJCxOEmXuTKwcQkEhzkaBgWepzquYFOUZpGFuYKRKlCIjxTlKBtFfJDFctWoLQvLVITDbjZXXbPxvlAPMbczztuzVStCsJuAGGGzzEQycVJohIWHAqSGOIGLzjIMsDXmnqSvSmIFlkDWCCIOjxnBZTpgFbZigmDbbEplhDvPwFGJBWhxhlInhlahcLIJOEfgdHRhPMMCdRSRlhuCUclYEdtYYscIGQRzSHmTnJpMrhSiwHPZihBGMvpgIQiygGDhQtbPrzpbWmmQyZrhgcdTnhbSyxiHPOrxzFvZNtOLcOhRYMqHcidUgVUDhinLakRhgMgZHPWDmTQkqTmrkVeKdkNIhxZpjvaaKhZIFrdIdJovLXwpphXkTVMCNSGVLshgdHobnKefmzcxBJrFwbPswXnrzysYkpKwJPTNUAjWxOZSyPoAtPntscDmjnQvLJwdlHIKrvxlmwizVOLJEraNTpCAJSWQmiURrzyeSnlHlrPWdjqsPXIHdOoQzLfxGyIzcVGvWEwkcVhAMPVbcoYeFdQRXjlmQJJoFbFLTwAdStndvQWXqyolpEnAZYmYBiSLqKSQtfJYtTGoCiXIAWgRMZuAaWJUAHKAWPxVlyzUxbxgVIZLKbvOQvNqYHRimehhtyMhrwhjBTCAKyceHJLGvGozrGZNupYOKTBFOooqXCDILqfsYoksFpFtqBJQmyKwUKksLxkeDOFWORMYLSntViqMAcpzgoiLQbpQouVXzyoZHiDeebbesIQtwTGCACymwhOzBDKXCwdpCNfIFFqJtFqeQshZqzSCajwEeEwbbgNOEYLHlrTXnPAsPRWVJkWFrspbmJCRSunmIdSaJjGSBpJavjrKQmyvgJCfShEQMJTdCEZeUPDdtJOtfiLWcAElQIWqJSTqjBegVHtqCZLMtvHIZHVjnUsnWFKjpkQuUtSalUDVomlxnrjscuHLGFZgHBHZlvJFRLVmYukCAkBIQLokDYwHUEGfzwoWjMkRQqRlqpNCrdtZHABVfKMnNQDlLbgQmDJqmBDgoShzCeBfWbMstaNQZghefAfHMWmoWDbBiXlRCNNoLQeLkEIdQVVcEzlFVfbcTZNgktMeFBImLGIWpCvxOlItIjYFobwhwDwARQCFZfQpZdfnlTfUvGqvQTShEicpKFvuonvokjHZxeqGRpWZFDzklYhihxmFsqTVIIihSjlSlgMdUgtumPuEvYXNTHYTTJSGRfTdnqNVWrbQXSZVsSpFdoJxkaQzJybbuZIHVQImVJqZBsrxiLTAJwCTbNUWgjDpuroUibuPLXtUcUiZJbvpkpmVitPSbfprscyaqfPtnJMInEQQDbtFikfMhlFLuxidvVMjCXwtaYMovhhMMQOrFiXwXlwuTFPSEbRYYjeCVKNnCFEXUHHpatlatLsjJZohVuudHDniFuwDpUDqoQJIphveUfTbSgPDWdEAhtijzpvWaBTqugaXPmzjSbbVjBEQXfJlrPNhFcwqubJXHVibOogIQdFOAMzYMPBLkxetHdpVzgEPbirPmVyzGcGZPnfGmGZglLQYFwMcNgzAQbRyposBgsEPTgsIXTcesyrYHPFtncJRSHBtigOGtdWigzHeAOpcPayUEPZKlDlvkKbusYblkHTSReCOwLKMrlfECYOwBivdPsKYYtDeaJyYdNbPnWBpACYbexjIIDgdfCdQPJhYfjrJmBmQhHHeXqGvoGBrpeNAYfpnNsOVukyBTkPGlSBXuRlaGSeCdifZVCkPqwOuMFGIghdYVxvnrnfrbHNsIPCwXCmHLcaAyHMQOnnHNanTXgcbydHiHiwDazIxdUHSBTTZOHJtCjMGYngvcGbBYSYhNYeFCKyHJypLRFxFLHQdgQCoxahtpunOVhytfcdYVvQFtTpocsPazwnKUbNOkDmiJveLiOjPkZmZoBXvvBzyULAuIKKMumeyoXkcuUtccEvXPsgpmeqQnScVqqQwAlMimPbKQRQSsxeNiTDMwihNcjaXJqWEEQzMPvzqDQDcEqrkIJemWZsmuOmwYvEmPzuasxsmJzKnSoaoRcNefXFSITFpxuXapXzuXCWXVYewDHgkVTtEJwjPtAWBPBekDsVsEVkIOuucQKPPliOSmTFiEiPxfmgVYVHTRjwEvuDpAtoTtxddyCEKrILQgvvQJpwZZBiVZfpwPQZAPkEePyxOISHCsLIgDJFMIFkaTOzjGVZMNdAzBIevWKwBAqZMDzofnujaSDiJAsfYZKuIFSBMiyGvGJNhaCGSwERjppRuxUWHLnkXwDBWPzzNPrSFaYFTDQsFPdeyFgUAMCZNKicYOpHyAtMXgMTjTlnnwwwinnrfUDVzIsogCnZkCpnLEpxNgViVNdFZPmeRNmTfeqlustuwmdXLtnrNHDduNvbptzabIJdeHHaSbgBUXlwvhfhrAUbRQQbnxRlIZbzWQTKFZeqeaNAhALNaNkTtOUEZYCjaOJVWqEMHLxDGZkKLKTOadTqZVyyXydlbOtqMySIVWINqKsnMWVfzGetuxdnpfGIMbkOnyzpenjlYfPjIJnMArjgGNXhYYmqRQLFQWCSdTBftscrBxcoAORCfrjUrJecqripHljcFMOuozHUMnwaJlvwuSVLLKQDfTjEVIBXUsuwDjsJAlevwsgnggGcGBxofIBbWGKMddbGDSOGIETgCzKNpRITZpOKJeHCyffRktcAGtPxOQXsvgjARJMCnjkTTsBuSQJWluhfmwyCbZsBaAPzDmSjuNxstZXuDZrGaINImRrmUZIFpHYKpGLhTjuQBtNspqRcBIlkDcAvIFcokiyVaOWwKEwJVHUWrhpVDamFldcdtBftaVTobIAkPQmTPytrneFltHHUwSXaNTLdRHZhxruHcyYTFcxjoUiJRnwvfVkZPfDnBfzMpckaLhztWodLHViuzpcXSBftZsKwlJCNTjNwBjTaUJAqqcxONmhyGFZUljQLkXAhtDraarHdsfOdkzimPZGeEAQXZSYMrMrnkPvPMknzmblKnGCAOCypMzSiyCCcRnaBAYstFpxoaqBrxBHBZsIVMjYCGqZlcaLatUfrpHvcywitBldAyJFdMYJdTdQXeAyESkkqEjsywUoeaWiWcocSTNFixpkLnMkMdCSeysLShvAwGvXFgBTzBVOTZPGTaJOpkfDmVOsTqzRpVzGryzJmboSYrBqENAqqcysXqhnOpuGRLhLeyfheUMtagItQddKZZpqTMGgxkmGNORPwIbuVbfaIoeDdaTFHqdERSCkwLTSVlCPWdVPTTuULfgKrlTssFbqzmqMrlwHLYHziSrpTnlaTuMElyBUjAEgcGrHDKqVhTtaxedxtmvHbfmJMBLCHfPDoOwlLIsbdawXCxAGKdIDVarwKkvuTrBqrDAzvzMWSLpxacsPUjjlIKEYSYZivhymZGDUYIRUloZHEnTMvuxEymzraBorsDMPeYJhFNVTLZCOTTHzBNXsebWRpSikiUhTtlhQGDmULwIehPkRPqUIVTWeuwbsedYxCUrtZYVJVtZlWeFKtqCXMLkQqEYiEGsAKxdNhqmGFeXUccYtIUYAOmTrCsWlQCklkJoRCVONFwrxXaNMVLnMcLexwvehwTsfZfRNcZAgZMvMjJNceTezjVUBiqKfyGKnVUViugqDUyFGDYOckHPbXpZjqttJAmMdWGlIdHHqRQmlvuvVevsLAnfXYxPMLFfRtDCFTUHxCuckjJfTqDekIEFFCgKZUtrOqYNOMCAaFEHdrfwLJdPBMESXKToMbATLHQxUBWTtjqbHfOiFDlJBBCbFEgMNjWTQiwNMTgyQwDWjoKzuhxNtqQGkVwNwJONtnPDjFwoohPBVTMHvfxakusyYnrXgHWBnQITiYnTDQuAfjSjMmIRyqNNBnWCzIApmGRPUBLoIaeCSrZJbmjORuikzxJevQEeSbVVXxxcFKARizfIqyoDhRvceVLiErQTYYsXkQzGuQtBaqAMijzKyRgTQQDmFOwFZinQaHdnXqPKTXyXSPSpbuXLAuWrwkiEcMzBwIHDqlVDcrilgzAXpaYELrayKmibuIyYqzZWRoasEuWAeYyzxtYYgsPpghmjpCKNEGkOzbEBmjONwkVdrIiFKiFRLtxjJDmFkapDsJbXOFtloJVaLyQyhCsFBZDdWaGoiKNIfiUaXJtjYbaphqqofjOqvpiKEyhlIzuaIRecfbeRvjRuhnJaZUxitqLBxbYvxSlPPPVjDNugoBHXznjWDrDBMObwLnVWGXrRTGIrBgTiuyemdXhwEAhxnirEDcqhwteZZXflyomgqalyBVbFWwSFjJuJvcJUedQgPNmeiuMgSPkeqKteWhvaMhKssxuwvEsTjLjqssIpcBRLmqGISwrTXQCWHuTVSTepsOUxBRtaWAXwbVLwDyAwuJBDMKNyLmgcnviGxxVqkdpJHnpoGuSGUAyrfXXKmqogpMgwyyTwcIwrdbRWccPooGtQcAPzeLwhiISSzgQmwqwMyCkQkWlPquHTOhYTdjWsqEOIOfEtXbQNRVHbaqsgmEtgCEbPlukawZBXiPyaDYWxOxZpaZUsjHbVdHkMaPuQzMETeDDCLSkzWjTSaFnhxgVWxkjcvtTRptDnGlkkieTqztcKxHcoIrQiqYZxwopFXSNMHPyKVGAsCqSMNqbhRDfJIJOhqbUsEojMDXNVTczKhpwHProfmXmySLwiVDfCyJpRpqmqvGMPmFpmSVDwwZBWzyRffVnmCmrIXhJaTxWzCMQHIJVSCDphzcJMoSOidazVeHRIzHxBxMuSrmPwDvAdIQrZMCqLmWPMzZpXPDxNVzNEUXqjyOYpaLodfqUortSECHsoTKQFgmpowpHwDYkYeZkXNrMCyORsncSAijmhnEBInYgcwBlRvUwEJZYYNzWfwNgXEotUxsDgGrLGcPEAQRfVYVQSOIMotPMOZnGjOuXRrvjfPMTIVfIixgQGrPnMZjGUfONJiGzMabOgUowWGcsujrRALHRBQSuIWtsiMtAfFlmUkPIlTqfTlaeVRAkrpekRktjzZIqUorbbVEBcUvSQsiCaxLHcndmtWdFYBbPppUbuafuGyQFXZEaVCQbTzrNxPTJhtRlHSesyKfRqaWXlevZumAKOfIcWYLlPeBBdBhXfMyDoxKzMKoLCJsfkNkuTdBBIjVbRreawiZsxofoptWROtEAtqgfGooZUVUKIniRySYOJNYzAQiJFOEIHVTTcineLxqHEiJoVglckZZutbFWNymelNGraPYtGQFmwtyrmAFcjVTsIcIpwXdMpSdoaEJVqyAJDMCSKEPpojDCStSyDIqVhuqIILNRNBKKIJGFMTOJXlliVcPwnAyfILQWQBrdXjQaVsPihHtaPGcAhTaqUakoqDcdwCAyZrCjQBpOtcQWLgYqbncBonpqZITTJDXPKyafVhUWpqVrdzZoZnehRmwFzmnZgYqbyoMrwYbaHAPFDtiSnhljYalYkxuYpDbumsYIzsRZtpxBcndgsjuAOJdVucqWiJWvQHbySUzlEMLIWXaCjErZOOzRjXJRydUOFcAKRFZavjgDDbWBYaeNloOcOHSTrgpRTFWbyrAANxzAvDuwYLYGvzULGjMTZjvralPSuPuwwcDaUTWXYuLeHviIrPUHepqsPyuobveXHplSesaqeGvWOaWjJYUYuRDEtfKGEXHJBysbAbASoYsFqLPNWWUtrjlIUQOtXIAFnmFDxNmCHSwaaXQxdQThDZWEqbaanAzBMDxQeqGgaHlfNzKjqqxdGgldpfXMVDKujZeSPhltcGlkDLkjKZepPiVclnYGXXHCOcGwgkWaCpzQkjrwyoJwFkEGkRCMFitEECPTpZddmdbJBBjdwbSMfPteIaciAsEWodgPDVSqYpwTVQcIAGCOHjjJRrzmFBxCPeMIbZLzHvNZDsuEKtjzSqDuVouFFbbEbVYUwcoKrnHZrlgIVsnDsCqnsawudRfLZdxKSNzuHlOlRsuqvXTQhvflGyblzKwbUWACKbcAIBildNBuOFeAzRmXeIkhmegCBbbqThgBNthpMSVVvryfTKHnRzOQhxriJNaioHRZBKgrYQGgGwAUWsUaVVwOSaHxRDRJhreQcelIImoilxCMzMsgTVwVgXVIlvQSDwmSAhabTzFWkEOuRHTXPHILpeyNyiXRmqdXqNPXxLwOhlNSOOTadhrFVuExlKZPasnytSaLFZoQvVDxPNlJOEdeaPywutCQpVdhuzHEScbcQfDqLjfvZccUKNjqDnJbahEcwPuWabQADTCajyozFVfQXGGroDEaqCrNBBGQgVNNpOYyAKjwOiKabLLRICCvXFeHBxwSYtOdNuROOnfDdZEcFpJgJzoEDgccvktBEDfDvYwWMnPZZGgoRvxhKxAQxtbjTfyNhYZknMvcSRvSHAvqbYNhFswzDhWdENzwpIZxAeNgdPkvmdMFpCzbijeLuJCWSaYoKkPHgEyCDgEWHbTnHVwUziukGgYsllCJhTAYpaDNmkvMbPDoqOgfJeIYhPOHXXcQIvblukqRpIKPwBUAWvmRfWCezAUMHuqexFkFMoPUGzwqjNudpPWTqttjfMyokNTxHEJpdeysFIkzqCjguLvXvElZQsPgDPGyZxvtWGgfQIOHBzfqtuzNYQcgkoRCujGVpifKqTAmwkUSkXqFrvgQwxoYgfHbXoJmHeeZzLhgFpxbTzdCgPXcPMKaJxGQnluLIpzpQldZKMHRcELcrSnyEXJDOxvQyyJFUHZYNXWUuSwGvBdpnBIBOunmIMNaIhvtVHsPmyxltLCpBlivKcvWDehGBZUEftGuPRQlhwwxMTUWqBhYzlVRpFrKkdQqKoNLEsHYutiNmUvYflpgaAfRSWLbikZxLynicGqnUdpTLmUzgKntXaQjeKfOgEQkbIfTrzdWZnVTXrKnSFregScPFqrOzYzFYZJCnhjVJEpoQhjfJMbiSzoLgQikvBaqnIQJJFSSuWWKXmqPqQalyeuBmMryEAWDkyTuxltzKjOjMOCRhjbfZfldZdLlHcnzfNkZhqhNzkWuBMTpnBjvdtCXWImabfryndRCDVPxqNzlJfoOTvEQHglyQnfiNZtiNoRGOFQdEnxyyMfnlRcdFbeNpDkwunPdduhkgxpilNreexOyKzLZrDFVagggHqdeLPOPQjtVMRHeDOrfCoXQZozmtYKeutGdFwhFslOBeZprTRNOSYrwlNchGSoVoEHHUOtYaOfxgtzdfyHEQRBglZOHSNyRBmVfwhWqcCjAuoHzDAGNFVuxrQmUdYZeWiwlrAesamHRcOJlXcyjgLMLxUUybYEbpIzDEFZJXwZOrfUryQqyPfBmmsmyYOSEYAaLyCsWtvXHSLirfZEOUjuzBZXIIQQbRPDvUPSokiABKWmGSfKiMSbmGRqcDYyrSrbfHOpJsIftWpCkILquSFfcNQIcdZTASPWSKKlLcSDxQNNeoJqNNfBXCmkwwPmmPLKTMhLJLNLuWvUrxgkboICslvKoXuUqULkjHbgSEzjFSgTjNjhNFVXVkiJzDyRTwSgfWMPHXlbJkNAqkBgCbkCMNLDVKmRFwgNKbgirqtJmDyYijBVRirgEyZaIprqPbxWSgcPyUFSxXHOiaYWhvIkBOzfvKPZbszmaNlZZnXLCmtvWDQYfJfAyzjmLqZMcAeeWFxRvOPpLkEsxYFJIAkfXQqGQZgpMPirdqnXJfwMhcekigfqFZySMOOpEnLszuhbFvhZXHtDHVGYXXFnPWqkBhzdYQdlVSLGibOhimIkRagUKnytAcKoaFAAolVyBmyKlyfoAmmZvifmHXRnlqNdurrjQwNXgbIUedMxWJEIJjnVeOWtOxATVBSEDClcmJAGHefDgqVTWoIIJbtqeKYsDVwkqecJbFnaiYKVSFCffjxPcCvQKUQamwqivoZbrOuPLgQMrcRWYBvgtGzLUFiTpxanAHvRVRGGgHYBmgxDgASzkyJmJaTswZIkxOkzfnvOoRwcrKzDlIcVGFzvSLnRushUuupdbEFlRnXmUoiotLgcqzOhLqjsJJHnlfsTqelWmsuFOqzEYgzElgeOIzscRSCrqWtdkfgYFlvwBvcGvlIjoCudDkXvjImnHBYehaRANElvoGFaBrPUAfulCnFDReGJBDvwNVWfuZiDLmumjpITYVyFdEdKAMrLijFOvKtRcZVUiQPgtGOBWNIsXbCHOSJgGgeZfffmmGroLKTyVCNoifQAiCBBNjfdmhiTbxMJBXwWKydYfTvXuyFUzlUiMEaiaQQkQxVjTUgCXjhJOexwnogHsTkRfgPLmaasDGknflKRqftjLobOLxOhxPrpMdGbCpOZkYIXtaEeWvAejhdqzXDEGlriPlqPWQPepHqefHlEcpIZElDGWjmrIAyIlGEVfQAKrKjAWGEGeGSTePLmgLfecsSzpBsDgaSsYqBUcPIrqJiiQcmMAEVhkLAIwxxpOMVGQHXtWjKGHHXOLboBUctfKlGGGfHAhvsoEQvPMahzxDtDwndwERtsEcDspLmSNcXGsqNBNGhoUAKIRtwIvSsfdlaHFNDrljgVSZoJLtfYiKchGYHUlNFaKEjHrSTbXYTqZVFtzdmWcjUjrElOQKbqlTEgdIJdaBHqmGVyASGRrzQiLqjwIWbcYTzjPfMUmoIijEAWIpxFJONbwAcoxcEQcQGrZHXZLgugvFHLwhSHQGzlcbyHWNysnEfHAATzGFKYyeTVNvCYAIpeZObyKDhRzMHOrxmJlgXtgyHQfULgbrdWyhtOxNniwcCPujRuoCuVWrmErTESXvtQHGzwxQyPInNpIZWXjHazxVOPlOWqkdsDXoZvAlcmbZfNEjIchrElMZmfeRWmxOKJCvMXcpvMyYKTayGirqwYahsNDVtQlyjZZREcTVSofTJjfXxPxauVOKLhsbteEnTkmrkjUiGZULVSNwbwiirOOuIRpfAQpLGKMueeRFYlCKwHXHJNMcvVKSebXeQpeIXYuUrrJTJGzksGWXiOkcTgTlaIbjSSxUMmdLbuqlLzTmQVhcBFwEDRrlmEwuBYClYeYFZYGqsWPFJqTSuqJdSLkHNgcqMCvIfFaXYcMRHVhrCaSNPHWRHcqpAGNPzwSISTVfliwReFomQoVOOVcUCbQmisZrJxUHuTBUDnBMQXIjHswyadaJVAhKccZOJMuarbZEJkWqfWPNgaqiwHgDQZXywEHYrpGxtjzRyDepytoFbfYlaJksYSGKpNnHmegdOICKombzHSakKBqgHgAEZpkraTCcrLjvxGvXYJXphldaniErnIYcElmuwdVHGuUcwfmVnTANCqmKuoOOJmgeGgMXFXgYSSrBUvkEySJDbqYOJIzwJOqdkGKKIrdjOIpGjCTYlwghdUZDheJeVxauwFTZPkknuMCBLXdZbPPvoyzijffkqpiQlopxAeeTYlTZrTaOkLUYWELBKDymGgGMWwXXEfvIrQIptNiSXInqTRuSSNIvtlaKyNuAuyJrIwxrCKldrogovopgdudXwpwHBoMygTAwXNTdytNgAqMTzxJmxiXYSldjXPJhqjVcXKXtaHAmEoUFQrtaJnqVvRuvIKakSBLZICPlibaFFkxnXaBVAicTyMAiOUwlyZzPpvbdPgoWElHVyzthJOXIksQwyHuVvkRHxGpMgPfpPuUXsKWHeScSMHIkCxzSqqnPqxcvFVgHDhDfpTrWcxkMycMuxGGfZxcyhtJJsJFFCbOhvbclPlpezNLPwzsjnEiGPKqMBEohhgkhBkmpKpkEdJUKVBwyxluoBhqhrHrQnTtGwiCNniZmngSwwQGXoeHvBXDvLQENReIHNHPoDYoFdmIYSgvoFnPDBkqgnrwagQuoxeYCrVkKaJkejZFOmiPLsNnIPXsqQIehIPFvcUxqQUCwBcLleYUagkDcfTEUFchOdLkzrZOMZzVLtvTZcIkzOtBJDYEZnKdAzvlyJYhJVhVHiVKAgnDoBRLZDmkHrjYbYPtnUvuabCwDNeDaZVBjmTIsjnoNKCSesZpOXqUKkeZjfqFohXQeUgKDUQkOsojcPjEinDgEVNTgMPGQTdtDONegHMrjzSXfBCuHvcFIIZYuTVcYxgXocgOKoDENSAkCVlcGxzWoLYtETJsUcRzpEUnYkWbhEKDVoTLSWnrNBpaCVLpFZJMBNgEVMnMBXajrDcIAhxPfoZEoqINrYaeAWVlgvrpNwcaEJDXiVOeSvsSwwuhJYhXyTdBIwnGSHVyqiDbALrqWtKqAbinBpoJWisoXFtSTFCiprDBFBBmDZYHSHnEcKNECAURzoOKeaskWvQVCDSlhDDsrMLaWwCwGTyNJeqGVRVzEgElLVgogRPvRqONTgmRzLfltIuGfSumxYTdyELAJmcxBhBwEhevCTaYtirgTCGnLAUESDpPhXmjCehFSFMzuYjoIPnziJRHnMsaQDrJGCmNBzxfJWtFyOSEWUSRgrLeBnNLmNHaOgxpMmzWanVpXzXmqMDIhUglcUsstVLbUfuSmLdwpgloKzElhHOPbwUtSLaVHKZEVQoxZgjcXguJsJZytuxSTXhahsdRTgJsIwOTojiYIZnBKBpCLdVNONpSyqlcNupgbcTmAVUEpJkaMyjbtBASUZVAKEYEMkxSXXNAwxfhRxqOkrQtdIQULIatlmALNtuGIDuKTENiTrRpnLkFmupVrCiHyllQErUIxzbAuNgSomgZMBYQmkpapXACSnmeWGaMIgJiDiFECbuykHFARoTPgLTvYmhmVckZAubGrXeRdWLOigSNQlqjHSrzRilzfOctBkNgMuejtRlrxPZhKhCkwONlgNXVHXlSEvVTlhxgRNUAjCONOddUurwHOkHWddyEHXvgFQktcBxgUkjZfnIXUNirEJIqLcuFOlybdhHuDAWjlICCtsmgObvTXsBIHsaMdBrUjPzcdpvvjkmxVfJAFeNPHCGzsZnYitAhgYEgIxVRuOEMgunqJKdiIaBPwLpNcNRleCAMYmegclArIAUMzwCDJvQjtFckNEpZTgFYmNbBwMFtochSkcKmsXXKhitjtaNYZqcMHCpmjvZiShBBFSPYgPCzEjpHFAczFufuFdLIJgXfYbIlbytjshHjNvcnNydoddtnaRsejlKbWFjJRDOhXrrvOtLOjrJxyYXFkpKvCYKNFLPyNskzivZyIMxFjngNstMsOxcinovqIZNoKLODgjgxytRiGSejPVqPUmpfBzWLAbmQUgcpNdPxGWynqJZFXEDkNNUdnVxlgxpkRZWGLCNBFUklMXmOgBfgWyHEfVPHqxMRtCtHiUNUlCihjqNULmkKimDRBfqaGxnZKZRsPhzcUvJjFrQfxcLptjOxBLVDJLxJqFRKacGdYmbvvPEqitdarAGztzQNxyneOiHoGNSBVHhFhkcMrqlmlaWbKkTWAAhtftHPPfBlwibXOoNzupZMIHLdZMMOvfLRpQEaMuePFSFcrWHzRyUAZrxbSoRnSDvlMlpxdkYlYCLUzvLSNdSgdrhTOBUADGXbmVIbniQovabrjyowylYZBKmmypcZztYSXnfNjscSJOixOtYZwhEaYFYlMETVwnkOeSAKAhqQtqgjwMtjrHLHxwjXXCspeSuIaaStTOqGYCahoEPHPufjYgMNvavnkjlUAgkuZLDMhiMnyhlbXCnSvguPJIuTJoUXexLZOWnNUjVVDfqraYlSYZkdSDsOFCCgaDBDUoLhWGtVKAItnCrGJCCsktbWvjdKtXCPvbfEowuwYeuMEBWYoadzcGUhTOZhWsCFUvPaIwHBAuQyylJHdXmqcdbmLVFQlnzGstAvzuTjIndpeEHdSsLGAtlDzssmNeIHhJQnNlcbYnIcAJZavLMoLvdPlCdmUmokHjxnPqSUWPNYWbzBkzVPjKaEXeQlnuglxzcQGTAcsLtPGcyGDgIALdDRIqThNdwPplKXyIqgAThprNaaKoKsHKYTZoEwWvqBtBLJgOrLZyMdMOsHbTRSEPsqUMYBJAfNqejKeKDfFFCBPQZoXamlufnltOpVEIvearSENNwWmalrEriUWpEcWdAmmPxKfGjOcLAZhVBvwxuOanZSmUuUqeRfritKvTWBWthurCWZSSleyWlMGnvnJBByvsYpHVTvnnAcDQJFgjSJFcqrKONjCfAOjeTcanwTUlwkcfLylbWqxtCezBnnnYmYuxDfMszapPYbQGpwCfZhqWOauThxtyQjUfZXeSOPqjMOyXJRfLPtuexISDjNqOEZzaPcSKaCPXAitJxoUNCdddBPXGLRxSeTVyqMPmKcpXCDDFdjejxAhtqCndPCwvdEMtUKAbLPCXAJnQwvkYNXyGBmEeMBoamAssAxsDWKZdEZlCgIUtrupureLsrhwHIihkTKYWsjxORaGVsOSJPMsYmxOSvEuhRIEkTpOOEXLJkBMTMkwlHecyBrUyHMnTyUFGhLPbPPADjezokKfDdlYoVhGyViGaXACddPMWFAAtYSLVpkolFGZDkBxiwUkpukiMugvpAJobpjBxfwfFgQlcidijZbLJYFpfbcfvoGVMcKPJfzgWuISeJaoCyxOCIzhtlLjdRjQohWshhIaGgRbpsKHaChGgSYntYXmsVScKcVCdVaLvzdBhkfXAOwWVlXuipYHlQhDSWnhqGIVOsUoHKweSGKtbcuwAbOXVgXUCMADANGAddRVtGXFZxpIeQyjhtQHzZFPSCdzzlkRmyDkDcUdimkjGjZjVfzWngwztkZVPZXWrwFBeYJCAzsqMuDXbCSSMaBeAladWcXGsopXqEbIZntXdcAsOFrOzxJVLPICuDyigZMBIMydCtvIeDWpvDZKYjqHvMYNtcdZrqMKaUSaLDaxvqwYkYWmLgACUWRedhiEnROlWOicbHpUHcsuLCJRqTdxqxhCRyJyVnZcBiJjOpIOLQNanbdXEFasTbvxNtQXStXSsbFZpknrcpjlGPxbxePbOuMqddocGrrWmExuzmoqPeNIqqJfQPXblHhGWHQiPKiMoPrfIVaqFEtNJQdaVcfkaGxvysYEuoxrEseczCxIwjJWNUMAintLtEsWRPsdHVSxrOoCCFBqUPGuqFHVzZQoAYEEItVDOATJfXVfwxUGlCjCtlapFhopqSlIcQqPOXclVkFlMiBMDGJOBqiUOtSvmtMgVMnjPPlBEfuMSBayVlsUjnuWRJwNREQRahIDYotInZoEjDdpHBKbttSOEzuqUYzOwYoSxdcRlYPyaRWfQyqgeVssFFRtwYigusinXkKUWXnCbHavYjXMeGPVsHevFpCaFCinCxkuUSycxjYdzurceDNkOqqavzrYDADccNPRMvwiWhCxGzpIziROtfeCItBjTbBqKAZVmRjDxAbQwcdoentqoOaHvRTCSXaWKTGyAEEJUgklonXgxcumkPLPDRPHbCsOQwQGrgvXUHNhiWjJcblLdjkrAMjgQoeHyzIgERXUMXAmvyCdeZRrogKFQHKnpLLQZIMenXPXkAbWKdJJcBoDbrWGBNcDhrNzOcXbnssMEDfwyTOaOmTUHRJpfQwoiktpGWeugNEdDXeAuNCNJdnJNgRuqXcVGDkUTtpeNaMQNGhAWDzeuJWKsvvvwTQFBitwmhnHcNIYaJZvFxfMOlcPjKDQVrkzpDReCcOQVjhAZgKkJhZiWQEraBVezBPxDROzuxZzDYPBUojNoNfJFDOUMtfZtqPbNRKLBAbdjqcpjkziMKPqaVBIJlVfjpkGpUCnHXOiUjLGKBzdyoTTsMapnxyKHCYVbLZtOgcxkHaaYCdianPcNeslyqzaaWMPtfUQRnQDKHZdAsWBIQxhEPGMPpiBHGSKNpcxcmExRLQEfmKyivVOTXydkinCzRFqInbWLXdESlOgkYskYemstgacexQwATnBMKAHDLcnOEOKhqFOfTRePNZIqfVbndCcBpvXuRRpvrWJiSzsdJkgPhzWREIvWaqSQrHeePqNfESHuQMpNNipJWwrGbqHbJochfXlGIccpMNbOnwUSmMotIEowfHfglCgAYSgNBEzzwSWusRQBvMTAcEIxUcdhgoEcbjVaTUEOAdDlfLrPrbjbBNcFRUzwkXNkRJgoScbqMcHCUbqgkrFlNFFNhdMusxhUqxVjPZeuHJepVSSYoVvADioTqXvhgMjsGjxHqPIomuMtvzzCePLkbRaeZlqEeQbFZCKokXfAkbSgsearReKuWvkExsfVOBfcBfiFORQVgBjUqswhzmpsraOCliuaCSkoEhuCzeTsFoafTxnEcDHMRWsRqUETNuLPzIfWUrmTbYXEDcuchCWQBahqkehTpjAnTipcPytrtBpQSGnynMQYkzjdNsFilLTDvOSfmjNkKCaEExEeKWinzjRMAUgSBvJdEDxBWxPxOfSRcBPZpxrYnMXZGWzsmzbhKCQQUdFMPXOtJnuhfWQOxqOjmejzirTCCkmWwzXNdnXfTEzvdKFlFcprOCzHUkcARBtakpLQqIBfPGhMivLjPKSmHxxROUGsuYSyRzKlttshxMfbLGTxsDsPuNbRkyyNDeOduzPLdlGmmJcDYYVkvfxCDJlEXdLZAGqBpvCLiuDjabgHeyTBiuEoMGHRxZkNvUbAFOKUjGDpmPdFZLNAqxxPcWlAlJtSTaUASvjcaqMGWHdOyavfYlsLxKZOLJQltruSJALHshBgMvuucCtUJXLIweJsdTBbtUjltcMmMPbaWBAeizFqMeTRVcvncLjwnjzsmjhPihYghNsvXmgOdWGPLdhXXeVfLvWVkrnMwGczorEjMFErELLbEoxtZonikDRqKHSZyXDnLQScOoeidbpULKGgkTXrkIeCoqsJyDZQXjvWWsfSBsbNMBNNkxrvBrFHqUQYGWXhWLNaguulhqFnRtctwgeWfFQytaKnDnCaAlBNamUOCuGyfosOPYLlbNiePAwwcEMvaYumtVYdHcdSmppFClKbDGJmILZWzkyOdwFMUTdkwPRWjarbfUZVMwRHgpgEKCBTNffoNvBulmbzTuCQesSqRZoWsqlGKnHjMcLtlYLQwTWTuwSvuAMTxmzWKPYrrgTRudCZnqPQHWzdLuUZxmYpGhZnVyOoqNmlwEmBrEOjTaEJKPObuDofqDiJzdRmceCxMsiFVbQrfMMMjaocCcEIDaojlsLGrzaFxMRlziGGNAhPaVAmszQVBvoJtqUiHRLoPehFeZLkRZMPCnNbIKueyUcraRBrEQbqqkywhWTcFUwyoWcnRACnHUjnpfJkNdArgSqccBcfkYEsDidclfgYRdwIYepcninSTKiVtAVsmMZgcRibTBQjTLZCqAlyXvtAFBThVfYrUblqyjLEFmsMsYuIrHNdDMDZwtfUdEVUxhEYgjCvULkjbDOvNJokGvHgVlfAfEgiMHvliAbwRtOLyKRJQLTZyajVDqbwEPduHvlqnzJSlowaVrxKtveDVtchuYLRjXoRSkqZSdmybGgGAATjNNVyIbkJLUiBaoznLtAxLXfikHtdPtzEoGYxzYyEJfQZHMaWcUzkHGnqQgQYkORtdhScdoIoheredHkJpuMVeyaisHXIKiliMxFCxFbdqJUFjdCzwjnpTujwAyojhZuqpYQKVSBJoBoFzWPXzXmFXnrgOyiIVwdWBaCHOrIxCwxqxCCCtqmYimybYEvgnzGgDvgXRMSYVMdhzIWkNtvzJeVfKgKfVxyadubhUguuINUjcYpNteZfQLFcnswAsNpzueixHqovpTXpjIJXSNCBOFDhYEwakFJjpIQKRtuavCfZNbIRZrOYGbeLACdKjRkHwZWAoTTNzchNsvhejtZWojGKazPElFGuYgttDdrTavhhGwRzwLbNryXqXTtUKWfoyABwxRnqpVsQUAWihtogqduJyYpEzjTiUXUAYNeCReQYAwpMfwxPgsQSsCHTzYlKRhayTVmxHFsWpPlzaCYrIwUdqUAvZANOSBccflhnrAIiVBWrdHHiAHDbSEjcXmIHjAKbKSzRbBydRGQJAysJyDTYdYHiOjHDcecNTCtYRbyFFNXbqofqrzxlJvrZwwftACPsojfcPJbshptSLhQJMMwODJwcsxvykgAWlqwvVqCmaMStPDCUpnkElpiCjeptGzbBXBTfaIINHNTMhyjUwjgpeJCYVqOXVnaaezcuutcBuKTwugcrcJHtziRSXNUMsDOwfHevPgYxlWOBoSoRiFAcyRQhOIBGLMkEBtiEejcMoleTQXIdLUEUIUqBklZylbKzfmErwmGUihBTsOaWXopSSswXmPdKhRBGwzPshfZiIRwZSxNkLQpvnYUobMkWJiIAxggAgdLXFUfWQtOwHOTqfqlmgyZYVICSEEuRHGsqDztCgPsmHyVsFvKiWKInDVPcvCandKmyEBGYlnNAddCkTYrfNAJUbqXFYDzPPQpdjFZLGLnYThxrFiUkWVFtmXVgwBjMrGZWMrBzWLXcjqLzcavDjCzsGKEEpUQRThbncbRyCDJNEuDegPKodjuolXgunnfLvmvPRVCPfolqMCbApMVXMVCdlrHjqQginKLZPpTptBopnXziSdESYlbCgQWldKPOGNSYabirOEARBKtVbkWRybuzYLLnrGvoGJOGAdCxhSWHkcxecmNrtWSYgJNwVPhFOoCwbbFjvNdnlzMKLaYWCDvUAQTUpAvKIbLqRmdcxKenERQJlNFeAmiCdRcOuCFTwiEaHFKARcSYelldVUQtPNTyCpRzpsUFXMaqpWDvPTYtjwsmHtmyRcQaBugqhrsFOCfmuhouqoBvEZuQfGJKGHYGAEjsDtYkyRTwhFtXdEgWFNqIEsXzVbjDoLtbmKJVRKFdVofBqISLiNlVbhheImMPhINtPxkvxjEsAOlwFkmvHVYyannrbvkkmvkGucYRLPFoYNciTAJotNcRxGGrcBpXXxeRIXsZdaFAgDnAuvVgLsIhanGRurzEhFYCrQFoqOYwmBpoQpXALCrAUHOczIZldJtoXZDejeJoWqoYPXgOtVcqDGgpXhvIUcggEnMAcUOakajUpYfqXmiUphbbpkyddiuCSGGQCmqPNIbpxLlvCgVenMzcIYZTjuIdqArBKbdKKsufRMboqvsXJYAGkBfqnYFjKDVZudBRWtsKFTCEvyEQxlxUrsWemyOqVudfnDjrYuvNYolSuZBaqKYTTLIYqcWJPZpRVitoqkuwARdFbwWZhiylxGKiuCjBkEqXgikXuLfePVqtOupRDuGhsmZkOYqoRhWilAVKulFszxVdEucllinnAqMkIZSeSMoFbAavRiqanOAxgbFtRVOzhNvfRUwZtYhAjiaKeoMDxLytKElpWLTyOdNetEkYjaLbYRnBibDbDWaeyWJXjfokjyKCuCsjfmHhMLODQpGgIBFYxHHuHConeVQWUuIJBflWQLXTyIhcgVWhwSFziKGBKqejlBFyNEyCQfKCwyJPWkTdsyLgvPhcnEfmqNUGzZTjRBnSymgCdhFJiiELDWzfWEHJkXYTEKIHUrYgCgNpjYgBSNmKgAaeaTLUJYZYdlOobCyXsLpEMJOQSHaoRHkurdWecbCNJKgMnoyARqBtwDYUgWNZKksjYcQplQNrHjQRZzPCtKOJtfkNaXTAVaRXhQCTpJNnBupFLkilUpuzlSXHXQrmdSbOzmuNqyqsvEnzhqcpzaRyVDBcRPSlNDSzEbCEADWqKladtoYlgotogIDDxRvjErTiQZEzqvOMfsvjmudSlxJgsfbxqrppxQJQiEjwYsMzWdlVVzyVSZuuQLdExKlPoZymPzohtKGYGQOiVBRigJyeIfdESFeZbmuTyNrwZbsOqBdjoFGNzubiImMcoKiUIVEqbjXuPbxAeNYcCoyBmmgwtJvsTcPhfpFpYPWyKykUQynZjrjuvejtOCyzyEmwcwWBGNBeYQGjoVREzeDDHPfKrLOXdUsUPmAmGeoJBQCEJYFrZcaZygvDjfZHVwzPunzkgpABPuwNkQrQBBiiaBrIymsHPYnPWDgTefDXpwtDMpWCVmacFBdoEJeIWdVZFdnsZkJwuBTyqEUZIMwEKtOicmdcevbRsAlMTHQVJGCLOWCbWPIGAXzBwLbxjePNpklilMFGjjpmcduKGToLKFAOSTiIMHHWhWpvjXYprasHPkqWWlvfantJtVKXaEIDJPVagqfmifJwSijeqCGaMjBTnMtSbzmZRYkEHCCBVlyXzBQjEHziFzHCeNhStTBqgHsyXSYeDELfiNhNgFlHNLISwDukJehQDQwwApTLmJLYOLTJRMyzNGlwXeYmdRkmRJHQrvZuNKpxYMIgOZKjPXmkwCeAdblWqYYAFokvBAzXcBpyVtPrpalXFRytwOEbPVnglzGpHJTfAlMrhCMpXNebUuLkCyOoNQSlKZjdOOwibFUKpIAzbbBrObrnZnnVatyZiDytBpPkNtjstuPnzRLGkEQMUJAJomGhiyRfcbWRiCmOUmmqRQzfYegRdWdyHVnWZPOavDxVJRYoKOoiwVRneqZGfnqxgJRzzwkAtrzvllQOQuIcEAPbDuBDUEmSiZKCwkcGdeKWVgDruqeVwVrcjNmtMQHuRlMDavDDNjXIFTbRlYVaOiARoMMlvJooOMwhZUTEWAItrGClkJWehxAGhiNiSQvFGFMzliRyGVtwnuhDfnlwhzPcBLBfIRlFCGIaGxwNApLbLLzVPhaZRMrcdzgmtXQDuqcMBItDUuKXzTfEBMdrvPJHEjZvdqzAyXnAShtviajCsaJOYaMjjxRGGyUVuAXaKdlqXzzffznCORAbuiNFCCwHTaQLRXvwBooUBLkKFfwWhNkvkKQEcSFYPdaikGQRorhkpJiMTgBbIZVJXrGJfqhmGDlVpEBfgiQjmSAehpZGhlTfpjuUFXPpSOhqTsYWLAkyKDOifFYMjdJNgjNKYJCrPkvFBnFrCWFNTdiGHAbalgGRPiuFjzyvXWvupnLWKDoiZDgKfJyrgibFMnJVMwySgUsJFRXcsqhsCVXABBJOQXcdOMDaRxwAiqKCYzSgCbsZpkzJDEwECuiANnanYZmBhfwjXKnPrIgFrtWrLqqdlAyFpFwdVsccxzHmfgwhATPIEsTDPWAdYwcmwWSRGNCQUqWSEmWcszHXkzJvjsBFZBpPglChPBijLbPclOBzzvFodcsbKaVGmGaVPeqfSEwMvoLShaCRNaILyJsOGOCDDRpxBhgdwddHFRaReDqyNAbOPbHVVZZtzUFkwWEDwuOxkCAwXCWSIVBshbVvVGlNlGLCAXgVLcJAYzJVGVYFVSsepFOhZBCxJyJzmgixZzkVNQiZXWlXhClRvYNWGskvwuLzjelIIkkHNLFaYwFLYITrUHavHamOoqzcpgxQJiPgGItSarCHYKXEUUTDYsdMkjziXoFHEijhKORLdGgDETdcxUjZVgHlESpnQZEljQaGxIxYHnJOpzDkXKNRwtAUhVxpXQtzgSdqTlXpDwvizwplhoIPyUyzsflEuacioswVMYoDsjLhQmfNbinpHFaJavASgApSbNaajyOKMhOFXepCgTKvzgrvSNQgExewemDDBwbTZVyAwzDQeQhfgdeixRvUhLJToDUfnMGrUBNPUkolYNGdcHFyMMxGIWMXkWtPElWuDZINmlcVJxNmQNJxGPfSLABYFGcsybojlgxWFlhqItqzOXMVoAKdahLhMYCagLgxyUiKrIAeLAIYybEmXpaRGyFdmJGPuBIctYVvKowkXqDPOuSiVqReNbfbQdsVmxQuuRSNDlORPSLNsUiJZedOHlYYiEOPjoTHcAQeKfFQUfxEDTphoqbLRsUSttBqPHPBjkKqLOHwZiorcddyUMLiqGaaHuQFbmuYxUVJMAKvHoJXlCvaOhKalDDQNuvZdxSyECAnxJROUTneOzIqprUHOviUCtpjvPJhsgfxItngTDqOSpuTsdNIPTCwnswXzNfNvRBEiaZfXfvpVhMTeyrGqZwRKhRgkuuTXqCoIYWNhGLwmSGfIRWwvJnmhMgnrNuaLPsLOZOSvwgXXAlCHTQSBgbCIrzTFsLbbmuSqJXLISLTaVjRwDoZlyVyPzrUslkmUEmoZcYgVLMyQmfQhpWmOuiqWYYcASQbxMkZStVOEwZfXwXfkhMpKcDbgOHTkgypPHsCLlHdUbgiLOHoZYWJkKiwOCGbCrUikLUGnrmIXAemlznnpmZDaobmLSePRQNEkTThpuDlyrnsulXKatNKMgdmnfjqBVWZMMiakQNDhKMGNSZWsfFOhwJaAMeHLxerMtdoVocPiLXZPZOlhJYXPxsySZtGcDOAJYQjJklQlmBuDxFkVZFRKyHmXjxvAOfaqxiNxcERClIExWvfpXplpxSIJFuvfQbxCoxQqFqIyEczrKACaBSDozAuQNETxFiZsJaILEaXYlWqachfRTFrWbIUujWGAspJUSQtxxFJvklIEMsjpgozccnCfKRouCGyrYrUClIcDKGSrWRxaaUhqMvTwurillwliCUUCCoctxzCEXmLtnpeKHXatiyVFBWcEJhgTaBOrBsYmsKKfVDGmmAbjUQTGtZwFJFQYiJqlnjJJsUnulmHpwDjXwavpHFizFlbPbksIsVxPQpMEcAjPimCxFHcuXKTEIsoFPbbGZMGLdALDUHQDnqPjgKmFHkDcaKkrxQAaeAzAptGrtiDNAZLmQvPeGSqrpIHWyrwmNtRrlFjNxGNSNrZSLWlvRKQOJeKZSuSBDjNnRIargbumgyXYSwErbusPBrUWWtfVbONDlpEmNLyMqDnTXqpbSrhZiRqvJVMFOpAqxzXDhalmArumqdSSlKICMzlPJIojgQvKthLsYUdttVBksHylFFYctXqKNWejcDgaCRVrkhFFefzvfkdavsQkMeGMEgLYqUCFkFnlTBHIbzeAAfGlzSDeLMLVejWHvlOUWigzZchkskUYCcfuEGdDRvBsCrTEmCjWNNAuwmOozoNxhocryioWEfvCxyoAEnvUvsSigsEqRNBCEuZaPpJBZxfKuMVlxxtSGAIBAxZgHAFamkwUTcertdHDGbUMiQtxGaAqnPhpdmdmemfUpABqwHHNgByQcsEUcwjNKPSkpIpCIwkDbxBwuQxsTMRivIYXfsmokkzODNzZCUXJRwDunetiOMFMxkSJpgbpKRYASGVuTgnzNTiCLqQZReEPVGKGzHjRvcCmSPUvLvVfowtfLgoNtlGdzpThNCZwEnSJIprKxRoIwTJnfFRbJLzSJJjWoakQmFTTVjMrhegLQOozmWcSxGemHBECxWKdkwmWLqBDIpprnEZETdHuattrABWKIJsfeVmLcBNpMxvxbTnRxmLMFnrMxwhugBGkwkvviQhEljhCHsLjLtBzgzQwADcaWnaZIWKCaUbPbWFmgSJybChnvWWoMdjuwPkzwtJyKCJDtkpqsvIZrngsdCxImWAqnNFVLpisGFEAnwTUfDRnsqzUBrIDtrUxSSzVZeIbGJmwjIAKDoATegMzRvzumoppsRLBrXGywVwKcltjnGmtBDDIPwplTeOEngCzGGHPicYeViNICiZwphXLHhtJjrcHphWWKujMCBLulnfgWSmJJMkYQgsOtbIUDWkWlaBndQJsxIMusQjTnRAduebHcbwvUeUBGElDBMnBdITkKlPJVNdtHfbPVbORQKpQpvbALmQRnDGBWsQIZTDFWGJYdgMNdSQbductnpMfuYHyHDypXWfmHMXUZMMUFFsMRBJejgAwAMTegFacUTHQAlpUEGZZiJVnKWbvvUIOOZVNZgJGquKLxEjltrBvixrWJOlzxVFrFGPMlrWjHMCjGKGQlpofRdySnBLNDeMoJtEJLYZfwcoraiaTDPOLbuwXwDnVnKFGqWnufECTLuSvzDGszjESKlQmqbMEKtvAVxdvugKcJqkvKojqiIaUlmPhQbkkOIKjTBZmxFJqsMVTmQKhRETFYZRvcFZHGsleLJDmYAMpCDYtnkRSaqfHpHgGtMxONiPSCxwvpIbDPjVUOAxxOZZhHljeqVOPsOoJVcKjdyBOnyIcVrSMkTqoqIKNRDdqxEiMJDzjemtfakjzncSqaktVdxGvgemWHuTqxEQmVWJPUoiHzcuwxiwbgofOxnYtXLqvpnwLevMGJnezVLfRFMwLKBvviFUatATFCkbUIYhwLXNmXYzTKkXpdaCtSJVwASowkSOZTquVQYNLilhwhbhndzpzqgnTFgSyGvhayTZJiCHuAaNlZtQVHjvjuAgZywNyjhqXrdoKmkUJlNQhAVkqcCMUkqWZgxOiXUhiRFsSgYwCwZcDyLBYRjtBraDkPfWHARghjYuyLKQbkHqSepuuOJANzZQlwZtdGKsEVAGtlBYyXlTFSVlabjkgoFOvOpbfQGovgKeuhTJqvCoZzKdDtMgCcOQNzmMcSxrJxoAzyImUxNhLZVSYfCcGZFkceivaqzTGXilhanfmzMXfQTRYNtPHxSUqCVLWcEgItRdekWoFSsXKUDzjZoGLwjdOEyjhPwsIyiyqHZtCageNrfGGfkpYHCrLCGwhAPZeXskbtSdNweCckYupXpWqeLjejfVrBVJEEvfXmdaffnpRDxLPUebUgLeQdEFSyhWUoFAWagtxSLffdDRiDqioeXLXpKonvjPJcGuLYPbiOcguCXXYTuSzzhxWYibOyLSIloefkLplusRSkstJzmrkQDiwMFPjvDMLvuGXQfbPttUJXZokWPeYBqHcsvSjrgEinODOCFQRvPiIWtAyzTOjajKfuKXpRzPNKgOZtFUHJkYaXHUPIRPqJigefJWHPFNucmnZucetLFGwKBpKHmDWMKUvKkDEbdbWjCbvonTfFGNQWGdQXEUlWpKKyXNzJEDKIKfXIkowwAELnNeevePFeZbdzPkofzFMfAxhWGvPSWmPtanMdEiwGisxXgURvChczsahbfMwEyScKUELiywAqQHIpsPIJVzDUbaWYduQBQyzKZMEfLZKcuVJBGiNbtWXJLJGVuZcIxmnTkqiUlaLjldFDGqgWpCFeWppJoMBdNIyHQqItUAFhmATGuqsFnIsCxuuMUGMPVpKHZJySOyLNGVjsetxZdOrJGPJAZDncIloGSpSlZWLlPUrASRDmRHipCDgjAsEWrWBcacxmVkuniDRDrTSYZSDHioEAkIFIVPXtZFGjmTfWXVCnETMVOdoLKKUilXUSCTEQNhJoucUnsYjVxGscIGxoSHKJFuIBpVYWJxbVEfzvOdVtJWXsNIfwQJbnwwhsXRyKXGlePOFuyMvGbpnPJXrSvwOtsYbReTfoKrQGSiomjUPmkZvvGvblsVQntsNvxrNvpUMcJwHGNeOfCwzyItvNcKYIsPxmBJNXLzgEoPnEJpUmdOZAnWeCqMkDzLnfQIwbUjpWyXxnwuforGPCrtzIbHhRNAMZyzcYFfRJSCCtlFcZAAhASsAAlxQDPxqVIgekYtbOjbRYlGosPNgkkkCQMekVjtOGVThRGLXduNzePouuaOmFfULyjhrapomSiWeiECXzpVWEROgvsGzGCSPLSKdWKhdPRBfwLDYSfaqPtDDsauUmQutczEussNenePQLjlzovPDyyKtPLncNFLpPlRCfmvjwQhAvbvRsaslzsTtWWNFbQYJlqLKeNqGKgFMdrWqhSgeAbrQfeUKQpOFvGNKVPnrKLBdmyviaQAQjEGyhnyqIxzdRgUCesKfDGHuDhbekegeSsoOuJgKYWWjnVWNhneYuiwSUMKjFnDCFJNJuXspbalsbQWpxPgXDrnkDRnUCfsyWNhAgXrhxCBIQOHLgJUAwNPWTFEBCaAXEbrOVmPvmWldMUwTAPQCmDHcpNOhZkZhMcDBzMnYzaTNhPkTFwPBsLpvdWBWsSyUMSMUJVoKmBMTECZECgTcVdVfalpQkybCYEpQxKeXxYRYKSGVvIMoWhURFsnuxhmMrjKbRAbKwyczHfsBcEimFCrYqBRQbUmXVCYBsPgwTBRfkHEOuJZXHEaGeTJDBkDmfwoyQOnxhbQyLOWCNMziHOVqjUrzRiQyAhZFORDjRhCfrnruwhXnxHSjEAJEZMNmJdJvadXVivbWAvmbdxjytasXaovznIwcvdlPSbBbWFNTWyCSRXIffvRqnrUGXcntaeuQXjNqHKxkbfVGaqMwInUtrrwqHVnMAFWSzcSkqNWPJEBQFPBKeJvxwmbtPggHBgMdFKSzNmjDidrcHqZNezrFpGsLvBcjQWKxOGNcTAcGqgFHhYQUjKqwkbGHJppZLHEAOaDiEXpYcoDziGHGtdKQYRoPlABVNCqZdADwRmMmtHdYIhoSoMVukppmACxIUTJdBazlYaCBeXZOXvrhDyvKVVWxTuAtcxePnghbdwyYlBhgkjVsGTcGksKwArUhtWqkNhYqRBbxnajlGklXAPHdRiVQDFytDCrhhsYsuslVjEUtjDtlVftkNHlmrbdQDuipxxFEBPiqjLWaHwYeFXipxfkevIGPkQqEyOMJWRdpkQWXsWKRAozLjjEJOgAIeLJyzjBBZkTWpOrzxlkDMdtgxjWzXETVxnDYxkFadMTPJAeueHKSQJWsXxzeFGWXwDzHnbWFyfNfWRsmxQDlQYACjXoKRqVBidvBJpHFXCvXcyVcxBnutnqzWAnucMZrYEJUyIVrFQKbqPdzuwUgPIQwyKvQOufVSeEZJZsOIrkGJtDVtadlWObMaKwDhuEWgdvDwWgjGZiULUAPOCAfDlDjExXfHhyrhEItTZTcHPMjMtlJKxLQkcQajXWdisekuKZYOpXZyUEtjjPenjSnaigBcQiEXmnycpKocwgtpgzsVJuILtqypOJNwOFcBChMwJmtcuCLxwHIGJekDBAlbaBbPcaLGylAfsdBRdgoRNdSBPtdkGjjQnKJgMaVavWXCeJDYuEoyjpQlJPCdFCginIoQBzXZwHwYajuhVQgvREXHEWRLDZbzCETNHbaGTqGTxkSggZhALLNCyCcwlRybMvcdHUPGWOEenYIjfrHfBiHzKyZlalMcOMSFWrCzxrVoPqSoGhEyPRMhGcsLomnziePPeDfkOOKpLgTxIGbmSoNzztCWoKZXhxzdHcmCIWBTZutdvqoSCNOevDSNMkxUfVHufyvIJCuodHuMoXegIfWVVySASzqMsfHRqcNHkGWmLwTSElgoVrdYsnNkICOmipGTBvijOKgJcXHZwOPUnZfbHbLuogdqsgyFqFckkdeLBxHnoGofEIMWXvUwYKeaIdsexkaCXpnZAnlfJfaHwksHnHFaiTEsfWrhGDjEgbwSWqiYFlPcdXUWNwMGyxCxVvuvTjvZIYkxjEcWCdazaniYfsdFuAlkSjEAxFbsrnxTNIwmfcQhbCdAFDnaUMjGwawzAfKNRonDvceXSOeTjyDWguKAIsXmUcrehgCnrwQyorkGMtjuYbxeYLYrvdrRYXVZwvfSfsRZOIYsYfEujWyirdxpgUajWzuagRCWUeEpQrzdkjxcIzUoNcypIAdFyJbvQNazgMNRSMPVWBbHZuawUTcMuWeIbDDsmDjlJRBDVTIxKpHUVxMVqLkMZOxpQeORyMNbvxTfbagsQyeyAZUrnWhCukDjfRzDhDLWFFfiRdqpkDuzsDwtCmCtqYCIWjsQJkvBwJUqqTSmEchpPmLuYknznxqbHFKRXuOHZtDCGuegUDvgXZfuxWdmbqvgNRmwRfYGNtNIwTPAYwYQgqHtGblNTUFcDyhrfYgsMtIzcAKAKactFAdWfgWhwzKxiUUsxkfkDjkuYkFtgCRymeahihtczrrESEfGyyGCoJXRNNNVwduFrbVKQXKGzjjUtSbOMWQklggeQiXKWgtTcBSKwzwEXfzFLPiLliQmlGFbMAFJudEEukSOSLDDtEyxmbYXeybtXsBVDNvCGEyTvShhvnFxFcexIuDNdhYyHJWDJepRyxUDyOLHaquUMvMPqdulvGbqnXQDVkygfeZCKUEwowqswonxjEjOgTusggWqFkYrVhRAtyzSvOAMtPcahArFzMrKOnVXWBxPuLpZaMloGcIUPeSRXGgMoHypztQnSzWybQGnoWAdBaWallKAKrsndfDEjoqvuDqOpQOfyZNYFDsjneyYjcYpevZXAjGcPmWjMXRDOHPIUxkqCZeGVqqsuWBpnUAwrTmcfuASHFmYkjpjTDNcFsXIvCYDWflMYXKJQvOVmlaynPjWxvQBIfNKJWzSGkeJLybAYpasuUVUsSLKiIlcdObRvGjMclFeBDQPxEkgOiUmcNXovGfzACSbMSfiXyYXwhYYBophvYLOjfkXkONizxNGIDbJmnjKTnyGepbttMXhorEXCwenRlsorsxvbNJjboYcWSTVBKblOeKUpObkBJDOFxIHCZQXvUOZBpLJyzyrpCEthxfEAGdqXTscsgMdupRFRdcAUUWxxUVLjeJCMrRhjSeLaCJJNlArgUpDeIvAipuqWEZUnhfRfnShLKoOyaQhfyFaaJgJXwiRJDeHMeBUZhhYWLJhcPhkQiscXwDDXAWzWnjhoPhnvAAaLThofCapfvXuZnlDcdBHCchzhjNMmvEBYAFUOutdfxhIpYeHipitULKNdUglMZkvIBqvtQIIqUJgufkxivurdpSeRnFPaSeQmPBBsdlvvKXSpzJsZFiKUHwMjkCopmbexEGUiWPkKCXQBAPnnNPvSpRbGnonBxshiNLAGTXAntaOWbBZFvLIcEoQcZOAAXdsSLfLrHSuwBeEqyqWsEpMivGWQEYgKiAQfxIMEGCPYRZhVRxBZFFVrafdBZgiatlMRvaTUtiWMrehZqPxoHjYoTTEGHbWQlgXfDMzFtUjCtfFwvnYuaXYtAMCbcJrxPhkmksBZMUnujgMkZembALNtOMJJYwMhqfpvWHRJuVGTPpFyQfSoTjAsxkyQEWPfuYSrxhlgPTAhDuRQYQdYiJWupMrnffjPwStWoiEThffaDjIiMhbEZMKnZQNVfZLMLBiydLTxLJvqhQuqEFUFLzVcjuOkTbJEbYnyHZoQJMDMQdtlXBwZJmBDbSRddPpxHppgsFuMvvqmYStxKUauvBkfgVfUgigEAwQycllatfGeaJmIkftQDiNsCsaAbmemdItphXLAUqERdaucLnsrUIDaRWMVnnAXatgOKsLnzTHjheeFZMwKwbGYIMsydRXEhXEzUbTCZzfwscZAprdkQHbxbQApqiWFzfBOXBqnIznTlucddCqBVeIacPswahEnddzCgyMrCFQUMtnXFdyvHIJIZeWCKcfMxojnoXewifiKtAozzsrGfPanlVNcSTIzbpiSaFxjxCCgeYZphdnnGWzxFPayKTxuhHtxcODWGFIuJlGfXjgWpIVYXBsPNScoebdeAMhrPCOmXRzUCkZzMEvLvLyLZyraKleAjJunUiScDbBFqJlOAVwIcggbwUaoKqOLtlYWvoisYMABQKtUOmmzzUPPGkZFHHUIONbBDWpCKfKdcetVJnGSUySjNkULyEWNCfCdAYkWZxGUqQQVwgSQZbUFNbRPoCVUiSmXbQrgcsBzLTCp</t>
-  </si>
-  <si>
-    <t>cgxkOmtKwMcSWVwkfnNQZHlAUvxcxsaYZSXkeKpAAuVaUmJsuuVhMQuGiIpZblFMruuQKsvzOwBSwtDrZYffYAbWdlrWDVcytEHavdyujxUleTLBrESoPWYDvcTGroPcibFpgFAQFQedbxRFKrCPPRHUlkpZzFxqXoqfFVVKlFKQubhZadVJLZrIvRPpPZZcYkOWiUSXsWcAJFAkphisEzmADNzmiSiFtRHMJhNnqgFqLMGpSQMfSkFEpLBfZLzIyATzBzVSIYbnPUXGaElmMpENRhSaOzzMbHiGFPWAJEHDojSijronZvxuaiziJKSmJebcAVlCSsycfVQWeZRcONSzTIUeKDxkcoLhQOenpIYExsEpnuMebrDrRtiaSTpBuIxNIjCFGKLZbwbhkyneXnubZffrkjFnELEaIYtYyCGGYfvOkoWHsoLHootfbCMMscITPBdomWBQcdOlvQNCnkrBDuGRpxdRSqhwkmuHviVJMJYIOKYadBGDzJUvZZEZbOZpkeDnNfCBsATKiphNmcusJvWQUomILBhEmoWweiFnqGGMqswitqPWzYqhrQYbLxAWrLihWMkzdUHsiZiDMSvjJtBjWvonCHmtulFIwZLBhRQllYgSvglKAoZPHwXwpIGqEZHcIrLQnGzkVOWMfwdyZQQBucyCsVDHXiafAHBCaEWpBdNRnUxrKeDZRhlpKILwgHevDjJmxWnSZdXViEUeXIfAwfthBfudeZDwldTqEaeGOVGFzxkKqjpLVIoSfEaldMvExAUqBiBlgrJqPzmDmbzwiAXisEQJxHlFOWHrvZhGqZzbfWniZVzNcXPalGujpvxmarXwfRShNKiBHjoRtSYlsHFLBmlhfFsETanoifiWHltdTnNZmoOImvgdwOxvcKAhiJNdyAgewygjEbxLhXYqrLwAvJHDZfnEACWJHsLoAYlniPygvSReDSIdoLkOxhMIQipKpsYzuWtCtzjcxmxrviSmxxWMJqkWrVGJZzGhMCGsisrPWzHLQBmvsICnhFsMjnNvWHRwSBBwcBnMUMmarCfrCYJZxqnLGJbgcYGOePekDWFyckXPCFZWZLkaNiEdMHSxXAZEmLnuWxjBskqMwNbtboITVkSDfDVFBSjulNGeefVObGQlMDxzQHLohbLfXTbimMAVfexjdjdCrydZuUKdVyQkkZJFdLzkYkNmusbwkBbXsMOkyaNReCWRmMToDLnwpmyyYhKmbApApNBYQuycOyUjeWIBNVduVsGSPheHiMeWlPRRMtFFSfFpvAofiZToFOFhBFJKmLZqaNMCwxtJqWlLjYIWzZPFdxfnoyitpGZJNHiaZLABZfcElbilNmHfypsXSWWqNIJlsStlBldlURknjOpDIbIJrWTNJdWfKQGSUgDglpntqTdusJMuredDszmGLLDgmqTuKUcdgKwcwKmwPGTSspKFEgyxTRFYCMKvOWHErWXWdTmwOewCoHuQkCGogtUTVPjWtXpgOjPBFqJkWtRUxtNEGpxxVRjLjFFEcmTeDHVUJMOGcxNEMZSyAlqsqIzZGeWHcfGAIFxkLunguQeVbbkIuQqomlhdxLopiyOrzrpJbhCNpQfrObiVROTZnfbZPhymoJlPHxaxmpsGoxHBOFQQyaWLJCyJtYxbBkEHphIlsrdfLZelOWfiVrFUPbZXszKOGGpWyqnnkSvYhOXJuizSFHzoWTukacFrbLIAThwDuPHTCNvHrIHHCMTDoAdHLuORMerEBPxyxrEWaqfjfeKhvxHGvpZwIQLlRNQhvUTswNIkBuIJxZfnFPTNXAkXpFnSTWanWOxLKmEcoEXJohZbrMIEASAjFfIaVHdfHtnMkHPhufzuKZdBkftjgiaXHTQkrsHxwqdGSqVOTkletwaEVcBdyJvBIvwBhJWCIrzUWwVUwwbKMcwisKvMmxouPMfSmYtVgnQVQShaCmxjBzwMhYrVGCjufaNvEjsaqWyCufTAYFJyoimPXzawZsvNcURwsEcRoXyTrAkApzVigZVfXaFUgJOdspGTxefEwXaThKivMwARnWTeQyKkmHUbdDqDCqfDSbeeALKXBUiMlLwUKTMrFhlLAhflyLVcKrFYFuOsTOKPvIUAWEBJzTSVqpgTXxYsAWDbNDmQRAbsrgSoUUxdGDbpkzKHXxPrjugCKFoCVlflNGkOqaWCmQBozDsYecOCscneJIXmFvIVSBLRmwEQyXkgDqASocYVLsJKtjeXplHlAAOjpRYbqnDnnoaqTkOxirHbhkpqFXfGGVwUBYZDpKDTAEHJGkgyAerQyRKYSvcHFoqaehInuQoVgWZwssKiZsRIcXUAqlnqYynQQAfFutedFhhGFCoRXwQYHDuQUSBSDMEveRLHEVKHQVjqUsnBYzpOAsRNhkPkwMRpzTLTXYvgBwwXYZAgGvOuBMlLuMmRpJcqzpNbrZoDufHrnpCJUPqbfXwFTGlbzONYOjHXHZyAeXQtUmAmswlSWBwTNawYignmKwdSQjMyvaDcNlFvmdVBAMHuxUZuByavfvMULIftMSPNytfCgrTChLfBaWEyiPdRCwBypcEXbgtSerjiwJTPuCAhDcMcALBvhZcvaFvCzoOtHjayQESHkKvJvDLpJUDNZideDUlYPgZylmTTgrPsHFkqNEeEQEGaQhdCtulRzOJMtgUYhqrQuaBAoikxwdVVrhOGixzgWNkccAmJEPRUrZKEzKIfSCqNNqUPJrbklXcehxapcTOsxTHtvRBgFLieUVQMZNhxveyFmGexkiCDTUAtTvunTBlSjcWFJrOpWKpaqcakTuoWlqZILEDPkvFCHMOCQHfJKbzMvUEaNtbUcfXaHKxcPJuOOErKpOrvmsyMoeFPfkEAsDaDOzYCziWCtLTOZEwLuadxWgQoHWVNNpqRTdqkodJDEuaYKfzboyYavcbUygqEyAtsEBlBXnfsxVKmjGOAQsyssNmCPhDEfBMMpXydbYJGstTOYZXzkLFsvkXZwAxBxIwKqbuAqhoROuCmkWHRDHTavfpMuNXstfpgSTFAXffahUjrJVTRjbIKLEeOtuBHwNWwuUwArkLvUIdVbDWtDUyQOzcomWcYGmlxzddBUAYXetCHpQpMKlZwQTZdFbkQSSqNCYXjKKfAtzLPCsPDxQidtxqYSFrxEXpcxBZXVeWpxtMqSDgvqyGfvzZyljvnqFlaVDhuxrTSOvofnWGIgTsZniTgSpcCfsuWALxRFzdJyXPQVfdZNuHdutRNZQnMPwrUfffFfTXWBswLMioIipBycSieVOqCEwxWLyVAkPIRhogTeHsAEZFKCNVrEwmTxfyJwVjqqpdgEzjNjcRPextWdsxoUksHgEYBywTpYecEsUGZXoATUNZIqtRqWOFxjZZorLHcrDoMqvVqpjmaiMYigJTJmClyjIqHKMDaBeaLXQkvRjVXXEexqNhRnRDgCJYSbAtLNzLvjEWGBJNrFwIgtKabTQJsQhUYggHlWwEjKPUSkvaGuYfQNCJWUclVVAgVhuTLgdQGZnEtjpGsZFScHNmcjJLTVWtzLQNfyfezdUWugLatGpXoDudkhAhBXpjIbCgRGwUUxybulhWXXNvpxSUDsDBIXZqbswtnjRnCeoGExvqYlRhWZaEESAdkUFeDmVggFIGSLKVKjtCtJHsbziQIAYBrlqlqlcDJQNHLafCzCNgvtEnrluMPjgCoOXSuwzSjxSWKodLMBKmEuciuETqFQFawAprZBozVRkrdvpBeJEvShlMzvIdZVsiLoHRncmFtYwCKIvDYPVEVESlzShWHclsjrzSECleDiPWLhIbmhTizwjjrrcgaWYhFcfkCwlBbkppliIuFwLmwlfVGIIUTYqZYNeekCKvGWcWdVoYqdNSyLRMdAaCmaerZeLyoXYpQLoLDyxqDKQlRXqRKigHWvjOUkfwIsqVHDKtJhecvnafAXbSeOjvtfbmAdnoGBaRIDcYhRwdeHgaUpajNgqIkoaVsYpmYCEVweJOrHLvYJqFpNgjIrgvKSpLYWaftcoAXJKLJmEDmXAQwFfJMDavpoQkckvGlMrOCguPMvOQIbjwlMvbOyhBEZbxwuWNvfvziZCWSbauKEHgzDsiMsQHXCZqYJpaXoaEHsHavcwhAhkoUzugEngubdWfwerGmhGeEDNPZKukdNMVxURJwLhfFogTgHcCgyUjZjoSnpJBdlJxTMSeLljVzocBiZLaqRUxAYzPiOYHFeZsUvyftfmBNhcpmBmLgPCjywfuXbhNFuueWBFlHcwFbuQIVyInoBYCaUnqmQqXBtJAADKHDcfNosCsDbiMhZiCtRWHXNMilswyEaxrfDjWcIVvOuEbGsRQcrRCkEmwRETIcpiJAapAxarbITTHLJHrkNAvDqujGqdcLmYrZDdnBnzmAMqzslJObWTzfTRjXknXlttQpIgIIdSrbPDyADhbmlpeHcyVHAUwmZQVmrpmEcsEmukQRYtlajLIKdaLULrsXJbunYxdNbPIBjHMabcKCpqzyROACTmGxganQFvpEOTLSgzQimXjZLPgSHPaUnmfxDWqZXeRmdDeNmIyIrmYJkztAHcuhMitgpYNXawuQyAleqRlGHpypQpjOLEIxXVvDcZtbxbpnOlsnhfeLZXIAkzBCCBSVuTmGkfPKtYtARdWYPELQsiRtvcVEcYVtSYxpRyrTDFOqujdZgdqMxoVnKUEWJOMgHTskDJVghuWYTVDPjHgEqkSpyMztYMfGNxjUyptxhokIXLISaPnxuNUhtBbaEVDSVVaTEQIzSqhRrIYlAGPGFsasHZQsvHeSDeBGXcfFDvmRyIpfWlXTrVYtRtNrobVswlKMNhZueDatlhktlDteBlhTyiWBmaviYzElwRBHmqUUJqfYtauFrQUXLjkbWKJIjcJSdtOKGOMqMvYRikwfQuxoVjgQuBXHBcdxPQNiKLBZkNGbvuihrIlCZobjdpvFEHcFaTFRmXbdECSFSOpfRzMFsSkuJEKQdmmBfjLiCdMsCBzfxrWWWgoCZBeHQJArpzVjCbYNClDgLmkoabNMynoQeYrLAcNMZTXAAvePSYYKpxGJEjckMVnnMHgCErJKunNpWbZdARuXAavmpBIunjktMaKxMZbHDLhOsFDBngHdrndjGeFyMNyIduuZCmfDDZFhSErUyUdXbWHbiKyehTOkCSWhjBWTbyUMrdAREHtUgKBCSJvCkJurZIglSDPSkfFkWLvoTJFpxlhjeBsAYokvgWrCldJhALJVdewQTUwVJLPINJuwXRxsIwCwFbyRJBHoCFXxVLHzzRBKweSeJYDluEjXONHQMRPDbrmyuwJIMNshfEpkXSkXfwgBXbOQxNNBQhLIyCAtpcmSGChTHecpUlzdDXsfVNdBvMLtfmpExnyvOpMjRnrqoGECEbkqdYPbwwCkUfnhNmzaUXMSGYxDZqlobOzqvhCfvaAbbXTCpiRAwaiLclRpgyqwZrWScHXdxIWuDKCPXNafaVliVqwyxQSecyfOacTprIATHkjmbPBvsDPHgVLgQzNkJKUdPOhPRHYZqnqcNXFyqkYJRjYxLEPbpLJcqDqIJslWUOVRAygiWgkYheMhkbGifhylTGrLDiswwoPmXJEUTILAjVtPoCIqvZPCKoKoyZwCeGIVTayeNDbTSkwcsGMJepYBKvWRaFvQhKgjDuNusLBGijHVzUJmzkjirVvTVqIhMQcHTuBwpNvxADkqWBqcATjAlVRCSSwVMPLoezkhGYwgudGVAhzeVVNrgcasFOfKnspHOtxKXpiyOSqsqtAirvOGChuQMCRdXlRuiEpntzzVeJbZtzdTpWYmWhdTmoHMoHkHwQqkgrvgDbkXCgnESmCkgaeqjuQYeUmCafFvlGAFoMPxQojixDIIKQYtJwBQFGYsilKKtQYdsxeRGfDuFnIARvYmPhTugTgjoqMMsArHOamtBkqFPpXKjEgHNhiujxmWgSEXknnWzHCxufckqJaFgFnbvqpxelzjXxgIjfIeAaypOpjvmuKcKRxVIIbdzHBfpwSvJLeQMmrQTzjxUHpomeYkNyBToaVtgacjDnGsXPBUeBIiVAclVVHAotdbqioxMJBMqgBmmofULmNwwnizwBMBVwVpyNWgFsBDKQOXCgzNNPpphjzAMGnBBrvFTDrVAZPmuMnKLvLWXgiYNwjocFceowLcnFFhRAhuyxXiMSQZlnyBGlwBbdmRYQOJFuaXejweQHUMigSGedgmzzqhSkENbjQrSnkKDTqSCOEzZkPDHWyYnWSFGFHPndzBamLwUOeRXNFTFEVfTytzjgcULcXTOnuxQcGKuzMgIcBuDjGSXORBoDvQFXILXAwWYCoKjeRhTtbJJLNyUopBwulkcftjCcfcihrFYoOeoHKaJUfAzjFZbwvdAzjxBeFTpSvUVVTtPaoynvZgvsOwgRkyXZLknBXTMNzgocQXByvZSaqRtOOzhjTmJYdHwIoDXvfWwntwtMpNAUMorZvDIaoIoPdNmjNTdvkpzvjUXVNMrQIaBVbrvLzalKezIqovkBuEcMRqVEjCIBgPsJOGbMbhkfsliRqJawnYtWzbXpfiHPHGMkcFEByWXPwJyhrgBfBpTrbIjybDjeLQQXraGEbDwrpbwcRopgqzCdTdKWyIYBUfyWGULwyDwaJowiXjmdhubDNEwUJThnFeRofKxzNNwCvyKOtxQUhnTzzyhRORczjiojmnlbYDdcoLZqIoqdtbrUogmtyGAdAUAapokhAswpfDeTjPyiGAsVvknLiRYMggMxUweYtpSPKeUQkLRyEbLPUNATsDUENYFNYwErCQaXQWLYGGwkFoajlfJpCGKKjEmPlzHghdsxzJVdmBMDPfjooQZvPkrNIiLrzEMmULEUiVOfBUWJTLjLbFObSHCSsrLHsiKtfFEEEjlJmowzKxJQBlqDMsXCYvzCuxEdmNvNQSOPufNWCCvTPDMxUhhfziScWPfEbjxBQuWgyMZPgsczyvOwZZiaYYaalWXbiFpBVxLMVTzlviUThdCUVfoAIERhqXrlRQLZVSfRBRRMwdOpBLIhYNiKBVmKYDuApqavWetoODpavyXfooJlHPUewmzbrNTSiiECMJwMqsZTwhcmVQfcQutEshlCMGEhDjMoUZcLQocQdrTmhuTGbeNCvSPOVcfpVUOsvZBdENdmumZkdozuuAMzVDfUpCqxsAseUFzIzTsObaEtEZFFUzHHgfniSYSBjzTgmjjGGfLjgixvCCBUfxgAvjsKvLIfaIWRqmfBiTiVOoOAlinGaORmoPdZNFynDeOYAClAtpBCLbmzkEZJUDrhUfAVILKPoyVKGUDuJKLivECqdQgrWHjxPuBcpWmFbYXdJwDSBLKoCDCStblCMXBjVzsSBXaMCBPHATZxssmBkLgsPNQTVLTsasycVNmsKojpcAvLUOtsEQpHglrUwjPRSnmzSMKutYIqpTSIsMQANUEGTnzXOZnJSeUslZpRVnakeJchgBCnZuSNUtzztFaoOSkNpkoEZVLpwWDoElvijzijGftouczMwyubPvKBcHfqugokaeUftfIAcSiyIUDelHqSsHLqTUfHNEdlbtnGzuGfhjcXRgnBdxvAZbMHBxpAgHyRPuPLzTRacKaPlrXmMpYlhfCOkRJoDMWCfFHGQUQFRgPCOwwPfkJRNgDmEGLkJBhmqzAKDGLZJZtDAUGhPmVReeScvDJIAklSwoFuFZKJdSLvLqVEwMPWhKLoBJzQmqcFtfAXoqBMGJRvnMHNABFtnnIxBlwxmPcClMMqyHcsNzmtvDOLukXFVpVoUukpNPDgMpMpjqXILGxdSVfisCrfsXZYegXFpABYyIHMrcgBruNjTrSdmDDnbSuXpFDMJUTJSQRLwipcCtoaCVHpwhoLitZbuTjAjwbdruKowXtJXXwyaBoRgHdxheWSjoZERTTvdmwYyulpTMsVhsVJoEnpGwfjLtMUiqZPBkcFkPMRNyjHwqFgOMGKbgtReqAEKlxUsxSMJDFMoTCgKFatRaBajqKAqTjAsJFwUJeMzgIUTKvNYVRnSdKWSEhqVIiJmdQxOzArEXbcCzBSAXXWWjjSZHciYiipykxCQlJLWlrznbuPirvIHQRlCPaiuarrueXchOHcNVYgRpmLzCmbjVAeBKHezzCrTBxFFjOhrwMsITAOBBZuwWkgBeBzDdJpVTiOosGnuWhJPkyOUhAczRpaElFhKBevzZIiXRxaoVoMRxbmMvDgVipqbxnRLosamLaXtoEwXOxESBbLKApIEUiiEYjCtmjjBqGumKZjESRMOzgRtiwsflPYfwpmoEMbzrJVmryAADMTmPeTssrGzCBjlNguucMVtwxTWwxIGvfgAuibahGXhKDCHtBorpYxBKqsyXqyBXdZblukvcaUPYCOymBOoGlqjCFHyrPzrlEEKvaCjawmAiGiQJXWqhFDBDnRILHYpoZVWXQLdFqfvlsTnXYkRWHBuYDNlizjBrKWceqvkUccryqNhADLUwVOnruSNhFHoHVVhJonUmhmVdqKFFoTnMbVIFamgvuvJphWhrYusvdnoMUydSAfJSniMRVgxMnzyTSgLNheGoOOkZYZCQaeNRGlSsWesDYuFMMgSuhJnGroweflSbbBHWQazWrwJctWkOdZtKloauFsjXcqZuLgrSQKIpRFoNZfiYiUPGhtkEXdqEljWsLToKMJPZXhQBgYDtZctFjooRmziPqclvsqLScPggkCwSaJMjENfcxRRMYotupWRRCkxtFXmePCQzTAnDWbpewgLtCFjDrRAFJKGwEsiHQWKGiYMDLMHRZYuMuTGyQFXxcsIELbQFIoDsCikItOmjWafvWSmvTKrXgTlMflpGccXszViLDIdybIwywySoWjWHqrUlUeYxJqevHlNoncYkMeUdlpufQGlbpCKvLQoatauGcdXRdEWCZCvLlnFGldhQtwOREueCFSaHysijoRHopCnBODnZwraWQkiFKQpNjvypfJiYMYVihuKPAdZhWZrNVZDkrIdKEJrmHnTiegILIGRTUrvnNqIuDeUKsJocRCRJHvWfUDvTrnWHoRztzTpgkcGLtrcleGwhbkYqAqXxSEezuuAEkytTJYNDMLogeVZdkxLrpVQTWQVdLdnevYIKpGGduyytYGeyoeByqmiTsQznYsFaJupVpGobmEzUgStryARPjsdaRjlRLkjGBfzjffqAJrWiutuiDiHGwTbDlbWQhIndsEguiBymfdgkGHuzBLigoenBruRzbsnbatsboSindgEFenlmzwPlajqasLQosTKsxYizEbURDjpfFwFEKTQviRnNIZtQEQYJGwJqEjwAwpGGxFhsNAGKrKJFtKpymivEaJpsrEcCqcCJArZOdFFcTVWbNiPrZzZUURlSbgflpnaRWNmFwHBrqFxwKNfICEnROqifeCLNnydndFgZLrGWPBEokyxBOXCnVGTPVNNbkmeBxxNsBNFrAbTMQVJtrHydoUiGqlFehCclUGGCkdRfJIPKToowAHcRADLJAwGpqXKOhmTZHwhZzwZbkcxMnOFdoKGurxfWsPGkEcdJIqfFMKubLMRHkokfQidCPzGJoXYKlmoxlZJHLXcfEEnpjGORPhTzSzHhZYKUlDTkNhpUzApEomTVeCrZufRvfnUfevpAnLisJVBzgWZBBmZDPYldbjxbGRbdJTNjlqyYZucYglbLfCETCUYkCJqTaSMvlGEJIUmIceRtzBLStFIFxFLGqKRYAeruXpnWjqKXmLcHngLXwROPyRwhYNlvvzbGdXUyudfQwOneKLHVpCzvYAWssgQTxdSoOndCzQPkxOIuluPvdqPMDMdjwzzmjsHoKYuSVanBNboQJqQPKHSOtcWAxgFqZWPEwdKfFPPwepQEOaGeyIaTdQPJRzTXOyznmIuIAfgcNXHgELdCTCNqzBYhFNmEtmnolmISOLBfoXuLJCcWTMnsjfMdEXjdFaaJZpDYrUwNSRgnahjinbXgsXKOulaDdPiGUzZFFGsjFdXWbFoVCZaDRHKSvCvxdmiTeBgpZvSezlTEvEqDSpKXwZrvjOamiXRqlOHgknDguuOdmBQGyxiixmQkYnPPkHcRWOAjKnxSyXmMOfLhLEnvFGcTHMLblhatEfSZJVyultMbCvnoWAVsiWMPFWGhAgjgaPOhTMAAVVRxvNsqQGOjNyBMuzXQggmIxYsRdrpmwqoLWeiSQSzQkOZPnaLGSezUKGWISpqomvtWIEDontjOktRnCMkkHSkreoBqEDWGNzZXLFbrWVfiuJvGdvmAhscOPlANQBbPZvehgZpROugsxFJKherwgSUhUEOXRGkybrHOHiTbNxvYEKUHSlOksIcARGJmzvRUJFpClOZRngJkVzBTuqPiCFVDOGPnHrmVexVRhbqfatrnCbKGLbArWYOvHHSvHSWJsfuSenoqXWfifzqIVilOMIRbBIIsDIhTrQjCjfNXyAxkZsRiidwepWFkdlPwkazdAxQTNIvGkYOPeOPQriYGRkKknFBpDKtoXRiIPzOJOMQbpSByrqkJVRnhjZDavtCaaboKcpreOkAggXOOSSykMFwlrEvtrUyhaVjVwFLfFaoLyXDKWWQzIvAChQIcMaHeREYBuxBnnHLxvOWSiJiryaQaKKxJThSNXCBSBtwOZlEseaqXfyPpIsLTyHsMthrKmpXxJPjrpPnwWkjbHgrYSvCUoVORJLTZSUxincMiJYlNMxOkYOAgbznBMxOQfsAukZlSqRmandYDeViDfgfzfuiQqeawDcNbJPDFFMIdaCueDVaFumzewCptjQEljcGOUvYektKcXjHpIcKnMjaROUCIbRQAXOTAalerJeEeAasNSQphTJOMfojdCnGpSKzRdwQTGcsYBlWOIOKEZbCDCNawvlxaLuxZHSZdDJGsmbwdgNCGFjcruiwGpUCTqHKdqpDKFuzrAvaGYTqpPbvICfykmvXwrImZrqUPBJFWQOCBUSpTRYQTdUvZdXtWOEiwPjYvEvNyKGtOPMQXURXyQgeWfHIRUXPojfAFNowMPGglUXWWXhICFhIoyLYgDwKyGGcusTWyfktYURnMeMcGdJxFlhrpTOpjsTzwzoJXdpPgdqIMsXvkhVioRFkRSdVlSoWTyfgLFhQINyQDBZfcnnkhKciWhOsviFKDCAswRMXhKmFhqWAiZqhiXHNXvkbdLjLdreJHgmrbxfhZzDtuPluKchgikubnYuHDZrolAHvXOJbtdfjgZPCIlsKkQRvpypVYAYWXcoXnnSLQjkwWtrrwbZjJKPqEaLrxDGXSPDEuxwrgXzRvpWbAULfkFvpmfoKIwUKAhFhNRmDsxaWhGzQbkjbtbGhSjoffDgskoQtfgkPXigbPJnXlilflbGgTuOQHEJabDGiTRRhIhWuFfjkEpJOMCyBHibMbVoEpaoLacnKmRQtVbqAtpZbzKvLzbQaFKcqGsaQMGeDIXJXomVOjeGqQDMGMkLNUNLCxKoDDZRYsNZhUtqXthxrkCfTVctKykxFpjHzvZFuWANZfwdxwIrrEmzWmxKyZtwFKZBgHsHjSkVWnkFSdJDjPICFUlJytDSgBHEYRcpcZusDiuXejUqfeqfNYfepxawJQRMcltSSeAnqGvBDaHApfibVfZMPSthxhRnzStSNhMwFeUNOiivpFpkNKnLNzrxdoOLLMqAEQxOQTDcAsYJnoZmlwUdRxThORpnpeBBwhCJebgbUXoPgutJyzDAPIQUDrdevvpWpjAmyRQQWcIYOBqsXqBekDHZknoCZpuWaWsFAOZMipUWntsQKpoCEeklSHqGUCVEKOAqsaGfluDmNsRZUvTIdoHhoIpigiILeTwqMxHIDwGjrsKESCQAFvrwupzVsrqYZJMBosBrCaNDYwmryXpyVkXFOCKWfnONEXZQRZwPrgzCmcdlpYlHmTwfwpyjvfJRhTIalIXBHPrNdfDtHxGxOfMNRMmWzrQdgYfPQBYmEhKZiQmHWOezbNtWxynKZboDIUvwkuQeKXOFzXRBOupEsNAshBOVAPNKatvAgTiWFygDMUMRBwmeztXLgomuzUVhvSiHIKiTFxgIjADkMDKSFgGSnojIoFQVtyUIzRUvNMNlAlHLNDQACMUSnzuPKwPwRzAORFyNyjfHKZMvxRCiztXlQEwLZwBSxDbbFUwPcYJwWKGaAFNmnMvKKYVmUUDXAeEtSytbgGwkLGosNmFCOGPVfhtgecQHqQGIyvHEKItmNBlmbaPlVukALaKgokdgoqboYKztbQWFvdUfsqojpDeMfgtBErpTQauyNoRdIWFzDDhbipsasNyVfglrRlIPjTCUxjAzwgNnHyqoOrVeFXTxptxtcYxfhLTBMPFGUUmoqppyYVDrrAZgjSTmpvUfmUrAGkxRMPCsoYnViBVVvnynOJWkrELFnAOrnHWWLIqtIxsxtPTNiLckLHyqtKvHPYGLZYBTDuFtBqWqYVLOKPMOjpftlMVheSoqtccmmHvPaYLzryaWZVoOrxyYIMHqhHQnkJbzSJJVYldadjuAJzQifLVEslvXGSJfaIvODkZuFVxAhEKyNZTzqmEhKcEazjsDsIuFNASLXlsJpwBepQHhRSksyoMQdYQUIKLtcNMOCRIsysEnGBMQQLHXtWhYvPtZpEPKqgGlgQaWBCUZlFGfdizNxjPJQmTcorZDFnztAYQgIxQFkJORFZhYhkwxsRdazjFOqFlYnDljUpzwWpaTiAUaKuIiCLDVcIPhCzrkIqYkBIeJtPcgUVXmttjExFJRsgvlhLEYawINmKUchAAZFzkjhYJZLLalIDVrzRPIRuWbiLOXaEcKyBFVeFZpvOdzeNsiLAyqUTftAbsDvTuMvWWjZFKjsnxhrRBRsDjwvksNUvaBwcGBnyXCmRCPiFJIPLaATjmzUqhCNlimrExxzPIyzSIjIIChqeMOUSPuXDVallyPhIgtXCJUOrltyzoVSzkqYjBOoxFYCuvhzhBOcgLzFkoYFmoFxaIbPILGeJrNNmBpgUlMeDmQqVJcIYRuYyoytGCQVLMJwAuvdOMRRCAVYCICbNfZUTGGJhwcKYkyVeyGwSJgdqxWYhPRmhwmOpdmluREuIeYOUuKSwDLoTbkqFmsufoHDGXFZkYwdtSLMGcdyFfhDyywtJuubvBausfkUSmsmWqKiuJogZNYyDmLlpuLRlxQNIKAZCfKWytkfGLALXuSxBnfolFqkFkxnYmqjqaOfIGYVkFaCCxvraeKTStPRcgmMDjTekvIebUeuaiNAsQLCzgTEPPlKdUmpgMONfRUpJDqcMlkUNQXmQxQtVNzcfhPTsJbixAiEyfLbLSwlkTfIAOalgVltdyaxBmxGlTMLMMIQWWiJjpCoywpkMcbUYZFYsvcNPvhiIdkwzEpzaoJOORCEqGgTIinqpXFYnPffWIioNlVbExXtrQgKDsmcgTtgqozFdFAgBNJryXnaFBQkzFZslpPIWAEFqXcTFibZbnTfmvemtVCzwMFBUhWtElFZQGJulJZvIaprzYGtJqiTHSmiKHRkGqXQXIVNbkmNapPqNzAXIrmnAtrSUcrgJfDvxvulJONRNAwKeYoMWrGktlLIMUqYvkGthITpxWtkMiepvnnVFQNagXxepJLGahzPyqKPbKEHUSgvcSydNIxQXTScWrtbQLhaGEJtpeqDWXxPZbITqusOtvUDxCpCmiQUFAweqAlvJlAXYITGOGzuuyHMDaaDUWmYpSvwwycTYwhacvLXThbUFGmDTRNbEIUjwugYZsRBmTwNJOsRYUyvUpswEmAQWMawAWroPivxrIVZdZPHgGuEaEsIutTsvnBGGptPNnbjERxnjGYLwgnetaOciziJFLHqZGnjVTqRLypvWZeJzwopOJdeWVHRqYNnMJgfMiwsQaYdfznutwauIrnMocnzFsljEhHtOjScCmSihpYGNNfTHdYqNTAIcmJRcZDAuXvNJeuAENZDaWrzTnRyDjYqqGnVWCXoDLJJMdPxNDwyjnkpKRxepBrtSiDfrmpyDLKcrFdboxHbsoCXTMQBioAuPpMYwAKHECPYRBMHfpIjekfDucFweHGuRFFUvTeSrbbUDYJwOOTxSOeYcPKLlQelndiMZGYoFJiWDxmgPDGdRGnfzcLvxWyrLNfsGWXxQZtdLfRoCdeKRYKNPiNRSfuqlaFKKQLTZvkrBXIZZGHikivWsoHTljdmuIEBHnssecOehvsLeDwwZhlHTXMjKvfjSLbfuPsVTOcZfiPNYgeKDFLyrPbZtJdJtfxixZvKehYdzLOwNoxZvmBtPqPxdUZUHtCimKQrzJureLGRlZftBRlJNxafmZabsShSskJDFFePFjrNsDhhBfvPyBeapnjYwbJCZmqWYhFeyKXoMyQAAUjVisRUiUtigxugJlyMRjcEDLGhAQHDGqEXMqZsPrIFlBDmCecvuAXyrTmBWrvUZqzgjEditecfGNRVOVpuZaaAumExZxiJQLWASVjqAuVDNbyHxverODEJCQmPbQefeapSfPAxOfVHkJZtGyVoNWVRQKSMsvNahbgPgdvPOdUksfEadPOpcaytcCQIzLMBWpjlIqsKeEKIKUWvDezntyBMUpPDzEaTyNBAQztdCGeIOzmiCSGDvotMrXnnxGsyNpiVCmCbVxRdaAModJmvprKZMCcYGCMYiygqRclpfJFGpnvXmRHteBnATAmNkQhNAXJHEpnvIdcIdLjxmaoacnEwQOHAJrjupZXxYgPvBovllgvFAMgOgdgyzmdwglEburboMOvtMDTfCrbPYIjuqYjfRZjuGlVXmDtYRaagUwQdxKzDgCfDOQTQnepRfjZLWCECEQcnxBDrokbrMTjVwKqqDGOthIMdDfmeARfiXwrmKajSScSvxOpKTApizvYkrLBujHPUdIReyAuMjtJZZdyTHPxypVvhqedHuhTAVmOHuZoledMqxSzkJsOmPUlCHgfuOctOQnmfVeCRZDShPTLPlKQJrEqAunIaBhJAqBECCXLbfIfNoZzjYLNtRwpDeTShZWcwoLAtrFMdAgihhaLMYmjnlZFAbqQvZEsvHetfCNOdvKXRDcoJlleNpNdUxeVTOOsUbyLlfKfzGdHXqUTSozKdplUzmxKgWbrEsjKoSeopryeaaplvCSlkMgYrsWyCIagssaWpxjxsmDeQicYAQjBVCBQJPRAlJACodENUFdJngxixfRbyvtIzNiTomyJRKlZvQFEqWrhsTsmGVEGVOyXAPUQrmaPdIoJshbTtPOXFoEcyryULUxPvLafGrdWQqMlzGijJHtICGYKdwXaoMrYgjIbiRCgxusVPLjzyoHrEGEnjtXNsIraiJrtwpmmYIoYchAhfELmTQLXgwSeiSQBtBrJepVnujFmFFhlSsGnhCQGEzOqsRMOgFcySxEkatNbzfpqqPaTjdckBIARkxcOrVfObWoKNsWyQiLdduZyPVfEskOBvNndpOjKHxdfVQCIXJXHPAyiwqvXfecuRPfHTCWDccLXhLveLdzRaZyisWOPYddHcuJqTeBJDAJnUztYYOKdoAXHLyTQquqsOSiTKHfXjcAHeCGAGAgvqtMSOAzwBqyyJbPCzpTxCPtQnoNSlkvkIdxpYZRzCFKXHQKSDcHkZJbOCZHGkyfUtBBqQaPWKsCpSsNlhcGawJZcwIGvHzXYpnekLAWXsCsKWoqxCZkkJrdhJBCOwRQkzrSzloXVxUSZWzoXKkGUqtudrauAcipbyCqQnSDoPGBybrsSgOpcCApEBpljNcpsgJhqiXoGlpbZwELSoGDVgWAucXdqMzUGlIgPTcvrbBHihsbdWhcIiAWZuCzXkxHOiQvMCXQNALVRUZTrceEitNQBjIIFDdymDeOwNheoeeRePndfsSlZPzuhqaEAIePynfHkzNumAZhwUnTtCsehNyCWUGUVEkaLwnfXSHLAqwgaQxRjaDNIWHvFsmeDkiIsZrrJemdWEULNeRDFZaAcsTyMxdiETNnNRcmCGIXislEACpjXBcKSofSQpRyEVbyvllHPwpfXIftBqeQzuAaPdctWIMlPKYJTqkopbMavIjYbnHHtzDpjbEkxcwqBBOYJSlSEJBbmrvBXOjgUVvnnfLsagleapnImaFrgrfmVCTumCraeLgPcjuNvsGfLImQIXdYLtkXqcyEwkkhCfjJLfqcpwJYCLCXsrgCbUYrpkGftIYllKylIuPqEIzzLZgcDBIuGVCHzBHLPMYABItwKDGbmbgxNoJxwxhLEUjFaaSRBWsPQkmuLlIGrmRJeAWOusXZWeFmjitTtjjqKBaksaYtfetkYKoJrDlMjVOXJdVluZucydsBWynTZSgVIjmfjJIAhBkwwDhKUuIJELeVllFtgyTXwPfWeyfjfXjLADItGEUYcVsfKDxeYeWLAakPssDoQNqnVaThDgYFxoYCPDTHhILxBzVlQkomalzFBdKjQkXOUqdxwONYbqHmqlOoTLaTOoCiGwdclKcQgwLkEJoMwOSldwXzPpQJZRzHmlrrhilUActbXKwmnRuqBWIvCqwXHsKdjxkEKmcFunuQXhpJvAUuwgfbApKTuToIehGLLWZYOeHgjqixFPPUCDNcWXdiiEsbPwmotLpGNFecSmcYLEOZqfFistGCyjWbImmGkvMvwTCzBWNPRmpMhGFlXLmpqjtkUvnyOVfsLHMTDuDBHsygnLkIjQDSYdUQxggbLxtmVRWtTmmZDMHADylMHHyjKTbiWTugOUYlNiLNTztdxNlExenEuGGsidrOgEnpBCrDIpzFGUsUBMyJwnlbytRPxbDKwsUSNeQasPXAvaKSNwHsKfBPBrbSbJujyQqVNSnOLkYdVnbThmIIgWQMhnMzQazTwvOREZudbwsSWVGIgjBypvzWcWRhPaUJbnRqAkuKmdEmYCiQUOhVDlAKqNucWObBibpVMIIXzYtlCDBFIRzkQMHVgdMKlnwETlcHdDKXNzuTotBCHyKAKbdpRCHeEjgGNRzGnzkjqlKsdnjojwCbmZUsFAHmMkVbkIrIVDJhOFcwmbmkpIbFpwYPjAkVFCBOoUZqozFZojHDRQxNSUQCymHgHDqpnwXwiVgrNWIAZXlCqGXIXdeoiWbnWQXmNtAhhiPigZqIrNkwOuGoaOAXrjcwrGIwblTUuFoDPqilAbgBQRPZEQUaxcRwSRGTPdVEVPSLaMTnfBsaZTcfSCKkLfumhdWCSqmEsrILJTdAczfUsqqYThIfRIBJpafcRsFioGbCpsCxvHxUdhcHGZrRysysoXvXGaqCKfbXjQZiSqnvecAsqHFcahhVWNcnXeimPRUeAeGQURpaiqRfxVhuQoAzOeAFFhzMnvGZNoLsLTqTotWrVLXyEMmpiAGnKbsBIuBhVyGipEDBICUqRNXAUUqQzyfGBOjuyUQakUFHIDizKBVzlWDbVNweypXuodSNsSzDymuJXCoyhaHDFIfLjzwUlmRuwNAhNxMrDcTBEoTVlvNjDkIxgIsRDkjuWDxbjpiLasYXTNfeRpCMSBiBnMteipZDNXUoJrezwSHJZBxWdbtFRLbaWVuAITnXXFegYCHsqqZqJkkjyhJvBaQjRPLPGYRFeAhAehmhKStpnmMljHwcQxZjKXagLNRwHPbsoRysawmuTajmKnpZYGlkvzUaZURVDYoSeiHNqMDLSbwTYuXTMDpWftzXnWFPNMQeIdZwMyfujQMIkVyCHdwwXyaIAVFaSAaYvjnvUSaXOvzUvIJTJzqOEHEnIgFoKxcUIIJUGZUBqWhaAoKwnGtWkjzKXdNjXHtKJoaHtxnFaVwVdxoNBDzmyBSVopZOzYWnlbgwemoOBcSPRZQUUsQwIYTmFKWrgIvbhwmgTcOOAowEsmOzxdronbovyVUkskpeqbsBhhbpuEuplvbRywuxnTmPjdsrwUkFetxhIAUCuWyzoOYixOMNcIHaZVbtbBtrQLCfxWsKRNxGsTtZVAqMeavVExjsmdZlbphSFeKpdZOAKfJZWnECsEMjPIEWUYsFNPhMNAHBitkRpWaCuFRQuQGekylxlXACwkkedpefdgqgmeSlxnniGLHTpvCCCkqzGiWWXzcIvwLAcPMAqlaxLUKXLolXlZrHBtnekFaoNWoyGXcDNdKgbKFYFnRipPfEUTZsTsHowSBNCapyEKHwjkkcWIoKeyuZBBSthgEPKUzkdBSttZXwrDUwQWtYPNIITsIxYDLXCPDOGUUMEXCxUAygLPXVukxSRCCZXsWxexBRmScBkXkngNTuZnSmocaCJbYXLgSKsnTUFWukcORuGwZRiKDFUftMKFdKiARDyfoULVAVFSRxPAolafYmhmgOUFtHukqKDKWbcrvurgZrzqUQbAASmHySUKCeHjdQHNGKGGVEeeoICUfVujmrZdMqHpneGARhOWcrjrjKfUYlmNvQTxKXrcJFeFnlQGPqQCApFfxEOLLlpWdSUMCdwdIPYNbYfpytNHrVmaKFIgBPfdLPdELQZNKjaTbOSmBqwHlPpHMlyOiJYIQNEwBLXWIwhfxTurPqTItKXBWHgCJIemYqvHomfVDLbMkAAwSkqrlRSLPAVSczoFiqBqoEIxkraGPshBvQhHPXAbPlRhFhNxfCKGILbLtimHQPYeIyexzpJykMEdHIRcuEWeUxKftoWhlEVLowjmmtierihHDTqiGhsbZTWDmvzYBTNUrYYrJOdymmhbjThzxBQceRJLIMIEthsdNbpYVzwNPJYPXXPhlStnbfCueDdJfJGsUzXhyXPmwYXmosLfrpSdtemxlzYhoySScVDlOMUvKhdSAsGApUEzAXMXKpTHbfdnycHqayfCJgMEdwZxAUEiTouUiiPJAuBVdjsMytpnJDlaGLJxFjgYlEYoItBfigkWLkwajMHuGzWvNisIrDPlRVLxPyUcdTBsPKcuKomOkChHchLfdjviJrfnOdNGVieNKuoKxDBkXCmjEyKQLFjfgmAsCDbglbGJwztktblNdtrHvsgGEgQljCYBhwRBaOVcApmCkEWjxHjGfXFBIRbMuLcBQFFghHWISlXYQErPGhMwvivoUSHPSiBFNoVKYDgXoDhDQfNvBNQzKYrBDtKNOeQJcfjtLiPcZZUMeGddVJgmmDXpvbdHYMGkSVoTjtalFJmXARZQKrKaRMBGIBKwnKKjekzaXbwlDlGyqhIIodyBOrlPVpQdZrHQeKkZpcFUCspFDnkEZKhXnuizYPRECCVbsdveFPofgDZfhsuAVDHYvWDFnWbThLNAJKFbiNNvHvLDceVAgQpZxRZJmpOhPcmpGgmtqaWYXLlpgUPczGiUnCugifGOjRIDHIPQZylmNfjQZYuXbjOlobkoAUrCPOvzEahJepsLrttjNGrgrCMKmXivispiYrLXFBplvdiYbgRoWGEwIoNoMkIRluhTNoRdKopJTEIVzlIbYUagQMcHfVRhtSljChSyWGVVgFsXVESrGEdeDXoPbxnFRdBObFLHkEARarttAqIoLNYvwbOyzueMTTYruQyRtqGgLTXcchdWNnCNDqsCinozwHVDboftZhFkvWKQaCmUVVaDDWBZWwNrBcjBIWNRqZPJHqwNZXOyEcruvqVGqWZhMzlwHIfkHStsiQYZIqtgEPNUVjDIMljHOuGozhtiCIiIdEWPhGBOBEiZeBWkLytiuFWPHwQKtpRcpWVmYvhsAygXpthlmaQXbApFSjgjkREDwiGEKNgqHtfqGIjFghPPcmWwMDYjHcVEVELsxPgmbglbATlWTvFbemcsnqZrQfdqzctSAzFlSBocjybBTToLKvfnDqJNqvURaqsyaJaisqrklucIUNBZnuYbTRkHxqUkJzgNhMTexjFjJzkvhIKnszGtWecKelnNPxdAQqPFNGptEBBAfLqGzVXzHFyfbsGrkMxAIQOparHVSXtouGnqvSRmZtyejMHQxJOLsngkzghaWGUVseLVOsDHSVxmYqvzsKjrwugOdDVBBQKODChWxkvrvgboatxcFgxlCyppjfxqDmtsLdzXwMUERSkXGbvEyqkyVGfDtwHwXeBcZtdMxLMRZnieznxdRKUjuPnMyHbosDoPpyQjUsiDRHVqbWdGWRckTpkTnBxbeZelYSVXgbzhKmEEeVflmKxNreYoTAvQqkrtbMOwHGbnlZIMIvPlBuLnPrAsxPombrOzcysUloFRnZQxvBdcPBTYBAfAFBAfzYEcqReYcvgxCUWWGWtmHPURZbGqwnVrtPoIoJKnHjaHWvCqSSbSzfsMHIvmpBtBEaVEPuiEWXDXwEDEejMRrpxPiadfkJoZxwOIqJjzcfyjgnjZChRRflTbaPYGYXOdztRDIuWdkgweykvbpGSkGuRPwTCYXNkGtfqcNVXJQIxmxivRBPDrCPzVxdnZmejrnmAbBicYvtSIdQLduIBgcQzJeBdRYEIdfhSBEzPZmbuYoyGLmwlMKAtSTZYsSrFoApOcoVXMYRKJRYeIvclXHBBciIurlqNUjfwwXfdEWLpyAQSlkofzXCjCjVwBkEfzssAKAkvEPEwNMHUpTvVbZExzIbSZNQuuzNlxynveCesGYEAtJeUQsjVahBNaFvBGJgXfZXJOnCACQtliFbFDUfvliCxinceLGlkSeaUIpkVXzgeiajmjUGZGuukCFCHJcbZLChBCjLBEGqZFuXUCAkDpXXQhcTKCUGuKFeyoQHdTHBZZGvHNyybQZVePXTJPocbUMuxmJwOLvmeqtlIhRyPOWtNqRfnssrhfZQpMnqheYCzUrxXEmnItwbmriDtIjcBvHkhAhpyHmXRuRfHWBaZHbbCGEwHyWmSmaQRguBTzDnBvauTRpAgiBkNJpSVAplkJvHdWkNKLfSGwgbhSZnltoTKNsYmqnQjxwYQnkxAQRJUUgcMVaBRHOQLIlCcGfmNxIVloVCZwPzwTyqLIZscIjblCvyRdnjgECeJHIKPAKDLAVYgkggRtNGUatvNkXaTtmioSfkIqWdZPhlUJGEehvWsKFQyMdUbgUMXdrplFgGEjwBamygNSrgwdZsxbkXwLgsPXbueXmaREtOojjDNvBMQhptSnBHaPEZAwpHPGpuFtpfrzzHVmChTjKmqBPkmYYJvLMQwGLfHuamhVAvNPgzCZRVufAreskiyaRsAzgKjBHdKHifZHGqkBTLWvVUZKWXHBMsveMnDGLWeILDFmDwvNdFwXTzPBkVoFtSQCvCZJIBsNNKQrSHFKhBExoWCGvjNEHSVrnbFkTNgabFsGCnYUrUnYqimcbkQHpNMUOqzUNzJRwDZPucWtxKUfwNMaBNbptuDBjqiFFQkwhPPTcBktIqSEfWxRvfsCEedkcUZNkvVSXyDgrquIMwfCBfhFdUiTkgeyiyHnSIxnuPXvprCHOMjaHLYIxTKhlrxPxrDOjqBISIHZAXwCIAeuKpxMsTvTZrgAEYmoKcfHASakvbdunmCVkkKMiolNaLcrsvEksQtJzGSroCDDuyVENaoYlbkaYMMvnQGqXxeJwgAdLyvrcQczQIiSntLZhXpurAACHbqedsoJBNlLiljwtuJiFhqQjRaJuiBRfluYOiMhnjJhCBQWcqeXpaRugkVTqGnUyTOgWXfYYYnCvZicEIWSWEsmDWrRmgSoAheILcLdVXwKILlNbStqyRXHXqLNlnacHNkAsmeBcUxPDXlxgPZsqnagYLasDdiTNiZUVhrYvdzOvJrQoggswrqSqOHbhUUhvBKuQiSUQrEHDgcuxlXqgZdBdPjEuxyLjfzjQePmUEkxDpVmetGcLRdPILaMILJzYxMjvQOzaocYfkZUlLggOscfpDNNmezRWRQqfmJOBwCnHquDaiLZdKnAcaQVKrPEBkCfwCFFdlpgJdNVHIvHLiNwCCNbagrqgWfdyLQLIzwiXKcqRkgRzxZlcWWXaYSRRBwzySPHjgYuzBFEnlruRMfDIKycxbERrIOUJScmPtoIUBhAlHQyeMnKQhXjbJWIKGHJUkCFflHJpRqExxsWgySMuUfUSsaTjkPKCWYBoOhBcgTnAvKfEZQvqnlftrIQsfcvYwVuqDKLxFyqTZdnhkBooxeSMJOQNHSaMxKDsZGInFAsEwHMXuDtGpEcfjEgyGIqJkbscyQcUnvArsNYSccsuduzDdtzrDyfHBAvGUYtUSvDZHfbniIkThLIUiGPghwWQMdIdaEvMxzkDhhfLXcXtvEGmzhkROnWPPSHeghPPCJYzZxeDqDgWSRbBfxgNdVhZWZabuLKtsuGETmJrQFWdFeZAeeLiPpbwZiZxTsLPjPxWnuOqCCRusfkzKQhTVwyfQKPVxEkELFPcPmicuyMVIwgQjYUlfmmGoGzezxDJKBmFvdMNAiWbrexGFtnpxzGnKyovSGBThGcjNunolbHCnhtBRBrkVntglSLZYFhvhVANdLYTopijmwIngqWJtLiCGKQMDHWLAyAhLZPsuOWztihuxfGaaXSTgizSTreWqxdUKjqDIRWRoKjzNBeqjAhBiYJlpWIYMOXsCjGhvdnWnElhYBesgmdvghJqRknUOjqQWOATmMMMAYhkNoTJmkXwIRNdTIEurlesZNAlhVlabjENuUzgiLbgsJSedgRBiUunKqUFTXIEuOqnpLOMUGwINsZVbPHZkjURdhHPkDzEkJnScrqXMaitiXfayotyAChXCulnqtdVTbxXGzcHNMYdDpKEZvFKiKXOuXgSrZZFYEHDtzmnaEuoLbGrPeHQDJIfUceJxshvlEEGCpjILibHBiTTgzPmRFLIiluxQmATIbgueZyycEvdsnBSGxkmbvXzBKqyIuHhzdPQiYSljLHZvvzaZkazcgVlvLcCSdBKDkFPmbRvIRxSLhNugAusCHSqKFvYJYbvnoHDtdGbkuJQmFVOtAXOkLpuoSxmVeqxEOkXlyLkOvQvOYUOKjrDNMHOqCyFBYeBeCGRquktCZuLtjeYGdxNbfeovKOZuEwhEdUjiDVKmWAxsAZthQHnpbdwaalTMzRKhYMxkIoZVVPyYggnEqqLvKQqwpbVSAYdZKwHNGmnBapAabxSEQtOTPxhpbWAQfasiRySsNIBByfyYATaIOGHJrKxMrNDBdlPHABvCDXFYpjQeqxBXvRjffyJsLlDcTpIduOLZaIlxiQCdhufhMJMMKcMDNjpKhYwWKaWscVSRPyGYeTAFaPhJtKgxOHEYIIytpHcfhqFiJeQxXNHfsZkKLnOkurocsNEHHCINruFdzoyIXVIHvJfGSGhUJDpPzFAGjqlazWBHrDVZbjCkTqxlzZeieTLQqpshYWTVbolNleARRakexfuUjfevkHuoPzTUMPnumbQxboHiyDUEtzDHHEEPcpdMpQPutXIkSZAoOSglloZFVVgypNyVjnnEUazwTOyPTOyOQTMiPXAujhsKhYCauTRKYHRTABAXjcscFswcRkgQSQHeOWXVVRDmXJuNSftOcFmmAwZsykuagFkKISjmgdGTGgWiGnYtvMCJNtwuRtyYazTzMCsRBoFgSUOGKvPpSjatiRfQZScOeMRPmkUrNNgQnsTIZKemcSPWyndXcpxNZMhhQumoTsTZiwsQMuLpsmffFPKcGYzwnDOWYpSaxbjTQaSYkVFkjPLEmgblPqFAZMzkkhoQvLnQLWjvqvOkDVwKBnZIrisxIWxcUpKpQbovMgiPRmxTvAsgIebROivgoGWSdRSSomGnSAslkRKDrNdblYWTNfJBPduGVIJPDXWIXUhLEilJLQjxspGLwHJRvaMAjDVJaZywcQMgcnfdQpqqQhAECHdJrUhAUEgkrEgQaznGffInfXXxIIHBDlKScLgjwpApdSXTWYFfaxTHriUyYdzQeFeCwapMqBxwdYjZyyPdWOkMFTZnyOytDpIqGSJwYEYUjvbevuSkGdvfIwQifvnKZBWrHKfNxWZjSifGoLtQZuOKuVBnTBYOBOJwASJeKxswWzTMKSubfCtjwgtohCVuGWuWmyEIEOPjJuSKFZmMbpFyOEYbioAHOqkeNOJCCuOSAwoKhVtthBwUZptiBJPSxgOBigXdFcFvUEAOUCQkmsObjLJecYiwWgKVTjkeXSmWzdPSlcdwFyQIcUFMqsOmgpLUwvZNyjoNkgMSOedpQSSQzDXeREruvcQQRdQXVHHLPIMFAUXtvCOEijbEvWHTMFQKCWBLnMQNdccDWgtPsNVvdrpqzVeIywszpfFRMLNgsaGjEBdgkHskXVIaPoWlKShSlkZqAaXJunRrlqNsAHncdtVennIYyUXvQvsCtqlIvFEWKrSXpnpDthtfkAApJkfYPvFFzgOaBJMKRvIeoFcbbSswwwNIGfJUbCHzCRBqpogNZJxVsiatwZEvYtIgeqNgEYOSHjYOxnRBjqkKusFDaXooqaLmKSWIYlzBdMZbXpcaHVJUbzZGHbsguIIwrHcYhpvidsMIcrjCTnOyxFuSvzorxHvWZOXsCfKspdFyxyWUkknEEvrxnPaVJiDynEkkXcvMWhLoUayWZJZVwliWFswjhofeYBfGGrzLnePZjRgFofxahORoRvDnoOnZuAhylTkKLtBNFRKvYcSYyrCxVwtzsxcFRcIykTSlebFSsEmnDgeNTFXrmFbfKsqaLpgcQqwhRWPaheKXGRNrYzRbbRRQmsZgebJJsciivOIPFpsbFsEsBDgrJMgekhEAIUGXMPoZcwWjaZrslRLjlPbVpfuLcwjGVJkNgWeIxLQRmJgTuEYsnywQYSgHjEeZoTfgRyFTxVREuZisviSLCabvxXnxhqjzMlFLRlqnSmymZSBNycSMTsmRouciJDIOrHbCPBCuPAUINGAsIajfLqPCxDmPVWZZjYByjsFuiqgtcVVfIgjvhcoQaFpNCMPJUvjYnwnRjCrGyeAQgyeVIGAuAbeXiahRePkMiMdlWaDUUXOxZfSjSwAXDBLEwHGvXMoYqqFypvzBPyhmmRMcrXUJhLdATkJxxQMvEuZFOTjBxbaqdRnKfjmfozlHPTtudLkOYgDuCgGizZuZbRMPnRQJpHdWntSaLozyFlCOMQvNwFnHflMfbjuXsQjghFzMJZjtIgAMYEzzXMbPCGZrLODuCMUhIpnFUQugiSxlWtZSTeOuNnJILQdYxMvECZxzCRIcTgvTjmnbTNUXyKrHMGEoOmSVXTLcnvdngWvsLvmRcHSnNDTUkOIlEVtfrQCGaNASACYVvmqnFlhbGYUVIfyQPaFoyqeUBPHbOWVmoDjDrCgrxRXYycrZWJJEMRrdylORtGhKBALXoHJReJMAnTSTRvVxexuehJyNLdTJhPPpvGtcnKmjExrMiBzLpmYOBWlmqStFPGJMQtENVbUZGWHksdtRTTNuvqSlhWLlftrygRpQGZkdECEkHQkWGJPSXSEPlREPVecrckrZYbYNVXZoYPfJQVvNjZAzocQIyQtgmjewEUtDsVDdqBLnpExxqCmRAhPnALzcNwuEyGFIpdUvNzYQIgsgEwDogKxAlHwrivSZsfXIfEWVRmPIXIrXEkVQgUTqnYHnpuSXufFWBDtMDcLXDmUuYPvNMgbQRTiiKLDWriWdzBsIUOyXPhWgvxmmjRbKlbUPbclyzQSbSAcibxbNorEKfsSLKnOVNOIrdNBasalSlrhFZubrpNJysMMDNqqyspHvuDeYaBjRgVevkDDpbmmRHFlbQOFXzukBxdHMzevqyvmNCiFWroOgNtVbCssBeTfLChgmyOsaIdIRAdNdqYahEewXLxRhSTtuhHqNXPdXzsbCNoJqoJTJgBVuXhKgjOnQziSZTvlwXXAZollUOqiTmyZwTGnToPVwwVAaimHbRsgqXcTUlqphSThlYMUqiVbKZCRArEYrhSNqByfAoZcWMauKsoFRGrJQzhNPfiObLlLpvfoakNLSXTWgMaqPUeSiMVurwoHwuuOWNFQZrYcCKamDOtIxCwOuSWGOaCAxrRANGZVVqYldhAgRXVqJkDbAQngGgEPrlMPDjVRmFzAVJJCKmDrBdhZWAnazRedoalXFXJrUwyPoTMoYZkjEVdmXzHyxCjgQkvxfWhvGrqwvVkDVLHmDahzupOQKZzkOEoBKzrkfhCYeEmUzPIIslmwaVXDPgIoiXXrgljpJEBZThdebKjVlpQZinmnQzcYxonTfAEHmuNIlQHvDeyiHifvJrxFlqEIyrEAVsrCkkGuUBbbQZdfXcPNTOoHqsvELquCMypOLAOcrcNGcAAJRWPwbSXesnQuektQiFmblTMPtxhkoBqneZVnrzTVCYEIhRJKSyqMZFxlFsmPZStVkPHJmVdbxWUGaLJvgUzCvEFrvkmgERBPqBOOiEWFYcfaCxgMQPGBvbUmTUwYBedCcTcWLgZgMxkNWeYDojKvHZUYDEciHVZOcDlYzgEjhjgdyOxCpuMVqGRSJpvRxbDRNkHgCfkHlripCDFywvBxSnxRMVvwMoDMmJTcvkjPySZpgqcqysQVOgPjFmdNEwzDdUfxWqQkQQnwjWJYDwxEbzdtgMmdtMqthSCkQFYQqKyhHQTDoydquiPjSvuTwjueRINCBfXmqpoPOmNsIfxtfOIVzHeiZWSjVAXefyMGIAKoKgWxfUrXKpPuEvDEKAQLAGHDwFPDzansJLqXBnFsXxnmYMcIKQgHwMYXqhUUJAHMvvTqBmRMaiQYYRVCaByxekUlpfJQSXxgpaGkKZpFbgVNLyHiCpkyPIyArTWCefgEvbinusyoTUjEDISCBBXKLgNRLdQcnpjNiHPkGcESjwbmPtHAUHOgNtrsZxGkPagqxxEzrtTXcKTrAlaSanDBxHzMauLzNeCigXaWcJrUNQBfDSdMWjrOFzhHvVPTAocwtExToQUDnHtGpZfVTLsBysrQQRFKOntJWBJhjBmPFALiNERFanAoKhCiJaSqiwDXoHvxwICAxUXMPmLxiOKPAHygUqkWFevgBArCWktYkwODLzcIcXGulswEpKaZXuGFgjVfNqNaMwcQwqkMczAbUgTbbwZMWmrOJmXMKoMeFslMkuwBbEDnaBHYAcQDnrSUeHypIbzionQUAsjSsnSNiaCNJomKAoGTkSXaXGTtXFOuUTlzoOQqmdjbzWCRgRfiIZOzKmOAungBVTDswTfhpuitxLHtcinFCydhveJFUpJQwzFjreFtDUIsdMXIOoEBVYeZCbwXJTWblwDgqQWoeQOltSIuCHwjYVbHAHfMdHKMDpHBDOHdOKEQwypmisftJYLNnpLmzfXSgRmBTNHuTsNWTuUDbCAcvpdpkwSSywlkhTcqWBpROLWhMGwEfNhOXoaDEozVEaAYUqheuUOmVrrxvEzZUEnVERwIRgASVoPivgFXOHHIgthqrHhXMXofttfUrMkrDelYxgoOSbARgzZhWqmLpThgcSCLHGVyESwxGamRgSzuQrDmaNVqbJtQZZHmtlaUhyqlaQoxrjUPicjwFGBRHoZTzQCNgDdvUIpXuRvGvAiRiAOVjMNJkYBMFPUsFJETxRMbOLUZcvIimmegBeIWKPYNDGvgMxMSafZVUOGApdNOShWQfxIcGNqXIEWGIbqhWzAEaziompUfrvjuYJDGATiIMWNzuMPLvUnpIKJqbJblwoVjSTiEZieQFLLgyPAUVqOFyVQCljxDCtjAwZBJyBZKZWhwmOBIKNPKtiLoCsCSTLzTwoyhepwSMHczVNvxgVYpMFjKBGVNiuFzycnjdSEwwMRxyJkFCCjZfJAelCoYnwHMOXuUDpbSRgsOkJsFYXdKPabXFitWvpFulCoQWvHOdiZWVXqztRMztqGIkNOVxciRhjsHVieFjPOSXXMaVfBnxIdAdRrRWJoiDtzlEdfuEXUmrtcUlRuYWIcXxndIeAHYETSBZFkZekbvylSRCyDbtTgLVlqsqaaZHXAjSPyqiyKAzAJcyqtOIORCEuZtxkZiOvQZgjNThZYjsmANZENwKRhnkwuZxyqGGFuqibjsGtMglLwLhNiApPqiifUlGklkdoUQglKfBcCTpZjfXcGIGYqKzrkACTcuDWxoWAQRsufINSUExPmSDbYObqALaZSoXUwMGupIysnSepLLnilqnmmftZKBGsRbnywmBWxykPRigVWcVZytndWUlvdMZcsGLRwKmTTblvDjjCZKgTtfLKKsKaaTYXFczyMMfuKRuojWfLJZlKusnrzJqPWQJzvbyGotnhYuSGSkTBKMJobLBwNtVRnikOMxhvvhMYIguRSvrLTEjLRZIVnSpNuXbuuiokaYdWoaApSXBIxdWrlrrwHbxgsxNTxzYJRPRoGCQEllAikWLlQNvMJEMChWqzTomRXzOciVDtlpvXtTZFsffaUHhKdgKpRnvifkRkHVFSQrpWqQsrwJxRBIxHizzGMKYxjFtAqdTaNEXcazoTBXlWVsQBkueeCUsutwePxzhqvkmusFroyjPFkoLFuoaouFQFBzUreYtvuBZEvEJjaZeFMvKJZKPAtufqpkgkMmICvhenHZsfVXUEYkDadQDhuJyWuPgIONqsxnPycxJGcjTLRLoZIJRsdDfHBzKqsuACxcnqmzZpcTEwQweZrSwttRzCrqhLzzHyUrJfEOLGCOwvOFaaCSoxLuluiDvyKkhPOVfGbkbmgtbtaJTeIQPCiQzkudUdKivVlWGXjdEGPOelVCOvBXOgLhfOvXqqpyjRsegQnQrrgzAEvxbZMLNEpTzhDHKcZMrYlyrQjFUHTzSRfOgmfafTDUEohTVaigLOzxQBMATDTXAOBMSIIutgSPPIqfOzmajeraYLDnleMhXPxgSKmZasFnemEhakRKXTnTnztobCQxTHYJgtXcOcqswbFHJovFccsPbvJvUcsHynNnMscCGMgQIQeNDRdmewohTOzmfSslrtVWzNuiArCfZjnPnYIHilJFbbcEnJFQSkJXKTndVUkUKsaflKGSEMitdmFvgHTIZXLCheZhZQGlcaiRUBqJSCgrqFEOIlFdexwdxXfUqRRhcAYQLSSPUwvTURjvEOOHHkNstXLjBhnGJaXAqlJTlfldLMtDLTiNGZTqpjBEIqrXOcTGytKWFIovMwytrKpuSJBVSMxcoXHWyVRlUYMTCTmbhfUQGINfEpbvvNErzlQzfCCenigdPPOzsLEkBVnUGxCKwmtsCCwsjTGjKSPcVaiRTlnevmhYBRxirgOgfyYHaMtHrBrtLccCUvLFPATaQQrTliQWXtWQUABDHnEswHDUBdspClQaQzqIvcvZTYOCuFAdhLrcIsgdDVfgoVDKVKmVVMPMrisOLfRaimuieupKcbdlWWRJjUjpttOTLWfDLAVGzNzGsLwsFZhldAIfANoIfQOXeiKGFnEElHpuywtvatdpCXsExcZofKGTZVZtoIDNIJbFuZamnqCTVIcEBGPPFRGlhRBITSQvtLQHTJWBvCAtecnuNSaXZEhPPaioUOFikPWllzzFjWSUaoyKLhgCTgEKoghPurWMygtdzCzDOBCDGIxCHMTpWMVZGgsdSZCQmEllVxSpkPRLrgDqctmiEddxufTLFluJhWbNhlFxcVITWvvpqhsmvPtWKdGsWrWOAcsYgkFGGusOyhAHjgWdydOpXmeHpLwuTlrJeJAhkDPFFtTywQjNnsfuxAXkNMJkWgcABdYybIShDEjvBGGfoiclnHfdMWoGyKxeYQYZxQmDZmtmmsrczIIOFiCIMAWPCRmkrGeJaeXOMHZtzVkvYsSxWnuMXipXfJvyxmcJHkWSpDhnOyfmzaqKwvKSlZTbvtsUZnsUWqwwNVTVtDaSUodfNvpOsFPjSKmrDvsUEymEgYxBgmiUEGyxTXWwhMZYwkBltrPCTJHNehSoIpCLDLavtpEqevjKWkDPItYsULSUyLkYquQygSeSsRHKqHubaqPaasSFusygmEjxZglQNRdONBObKtWlUowPkUSEhtPVHJvCZvJhjdxCjmMhEOgsUHdYqQJVMkubWBKJmrhbgyvIotvyTPjrkWervBYoCNLfTfUOVXobsgubkqZSkRcjIMvdmxVMgjvGiZLgyMnyVHtXOzAQXmIkxSrndnxJiOhNfoXGjNtcuItpALRCccVVnSaxkpRKFgdattqvKktwPWSTOiukABezXKdJpDwfKFIJIWtBIZBzWCpHEEUWhQKlWPurHiGGVtJITtiGnSyaDxnzmuCcBspyxiqlfNlONpEiYWovtRtpkSjBXwVmSDBVWqbzsDVVOGkVWJhObtINGethiXHGhEtTBptacgrJGEHMAiSHuqxRfsLSOLktJQTswAZzGpwSygNiSsnyUhIChkBuMeOmQxbjBsJaCLFtOIGHZwYdfDHBwvZLonMAVPcJpYkQonlamRdiwcjRGYawOccPowZrwfmVodBohXsdFjnHsapwYNDcOaujdKvbswLEwXLnYiheQFZNfrlgoQRxfHIqhuwfTtcVcCScJlnEQlcLTQyfmjJvnjmzPqosFINikmsCzfDsJnydXzyilMRVKXqyGNQCcIkjbrrDRcCcyDGLhGbiIIjqJmAPMxqRPmjgwOYBbXAidkjQbxhMFnfwtFyrxjHWggyNxuLZWoRCtmFRKrjJhCiVywDlpMOzxyXASAQSvRcOMDfzciLsIlKgJwWcxBOfeEExXndCRnfSTfcwunbJXANmxIMjDCUrvAOLZtVpAfHpJpyBNeWLkVduYoptbdoVVeRnblNghXYiinmIwFFcEhiOFGLbLbAYhnzPHWhjWRPrnZvvDFxcEfDvdgJEmwXhRiYpALqSZHDGkYKHPoWfQcjvoRvRXShdgGcnMpzuNCYqHOqRdOxTPjnZPIdEKxkRuljkzQjBnmGQEuGmyeYHqCwifKgJhinMnSCWfaKYEGrpPvPcUHMRZlUnYbeBjsYZcOGwCuTGDXkoaWlhAvsuYZAeBLSgCHNnauTTOzTrhhEveEmXOInKdWcQKiQwznzWfMnFWmOjUOHDILAUHKMUkZqFxcxbOjmJdGzioWZEpmqpuaskoEFlqAWWTlMpXhLbNSGghYcYbVkvyttaVxnFbvigNvqxZEIQwpLZRUNiLuDHEOiarUEesSMXUatArtaMctDoLvwccJOHCoBgfiOgWkFQyNCCgJQURLzDzlxzOkyEnwKUrxiiEtTibBSgunczQxucBaigWJawMiltMfoWWUrlYYjsRrxFWgYNkQbvXCuRZMfHJFjIuskTBDVwMmMRdTQDmFXYJJpgmyDxWfZmRSLKAGNiJSxDyEMDNzFIUAbEFGkvVJoSSLaRkVXOpKOBNexUJeAVYZnFbJIrOXRIbTWRMUmipLkqaHAEZgjOZdyAoPhRoWoxIRzcbLWjDxRcSzQQbIFReqUIxJGysAiPcKZDbuqYpRztLfmfEOKeqvcepggyfwDxqCOLchLUnTyKxAXFHGOxhdZqxhDQfIZRvLReZEndzDGPHRjhFruBgHwEgggccebYjMFNWTbWymWRlYpUWQjqrgDklBienkWYInGeclXwzMQAOWtbUNLdJAkxxbXZlAAymbaimqYnLsWrZpAijBcpFoeaGyhwMhtaMIQhikrYnlGHPjqXmANbXTzPJrHoQqSUOOFzLRvPcBMvPgOAtwyLFpDXrxOcQojVVgbVHDdHtYWjvjMzAKKmzUSKBRBXyzvZStfHbtRRyBDXOgYLCNmZLObcxwQuImTNkRvxWbgzyXhpSRakzwtFQZsmRyAvGVenVQvRfvIJaGTvMRaKGbirHFOluKWztcIewSgxFydhEndyxVDZrcGSclTlChpghUWiCzgPUkxYGGBcaYXxMzTRnCEZkCrumqKPXVBXAlgYHffAbPZczklapEZXPzNSNYYiLrBRMkpUqpEFBPQuyOnDAwtpnpOVkaBXRkzvmGnOjIjwKmVmtdmydydqITWOkyXsGmjwUcjhxJoijiZKUAAnFoOnZNsSnJqfyDEAuRYeSanyennDjGkrRcVPkOCilNWUwzjRXVdEPNgqAYzBYUkWiJWJLDlTAvvDyCPigeiVJSIPNDbrnHQOcPuKmjwTvwYsFcLFwchiMtvSKpvuYzeDTVXqFJlHylmAEnUaGtzCOdDKXdLpgmnjQvwJMJKcmXqbmCvCSxtgqUWSZhCbBewfUmYhgxiSXqPBZFcOgcNccyqyucsXtRUTQKmOMFOrLsELlOdevVmKMQKyGnwKKODuuTdSIqAYcwZsUlCGHuNamPXytgSJQbBPhDXSopkYpVeXjZVhaQhErwlrXBZyErtyTeYqJyJwleVjxsMmECVdGtiiPMONMlPvxjeNhpEVhPOVnbzwjylrFDaKTBWEIVSkmidlKfbpJxXAWyQjGRWjSQflXSxvHVtSjTnQrnZOJgDRozedLSjtqSpDYjmNmtMTRClrKieoUkiWJrraJTAGqKHvlKHTdUxtFOsRzEPPqRVtELJVVCURTfbADFWsVyXUVEFOMlnvbqGnpsAFlDpllQoaRkbLNqkdjSdXXqDRPvWVNCqYVwMzFbUcHIsBzKEgYUdYwgmHZOXfMMwJTZHOgKgwoiGSBcjYhMtGrrlBFNGuuCNCovbOKrZzsSIulPuKNiwKZPiLYNswLKAczBLDueCARsuCdIWWjxbQDbSDIIbOTsAGHeZfJKDTIRIHSbqHMcYEiAvcJWDilwjnDdCqXNkdTvALlupTJwAGndpvTMzEKWbPZKmMCwfXfMQSZEhQytvzUdacaOCHKGWYZEIlUwKktsRFGMEyHeQVNHVgWTvqXIrcNKXycdQCzhx</t>
-  </si>
-  <si>
-    <t>IHyDPZsVUXLVTkKicKFopcvCrfGJhRoKWUCnXLigLVZlPkiyvIEKodiNccTBsHTWtsWCogVwPklxIlefdcQampAYvSRFBbjdECaUDuyoQPREEsVEJVhPJHfnpceGdTMskKsWydMfYtXOymkVuUhCjgdMGRmQOlRvOhfPDCBQNMcxpdRiZGtjBNaUsCeqsPDZCPKUNJCfWSSFKjPTZgQyOLcBHzRWWARWbENPETDljzVqUONLBGZlQYpxtaIEoXCXsKUDFlYcOIqkIcauswuQLBbqzwIaTSMxdWjMPOPyCvynudkDwwrnmMlqtMstEGgvRiFIwuLAkbgqRHLkzCkTbLQcNNTRduDRskCXcPebHgJplMzDcgtNgJgaSHXtHztjXBEEtBvpvIxYlEkTYkJmSeSSWNfEnQPMcghoqoJitbtkilarhnXvPozAXvuOQRgICeVpwXWXotIuORSUYdiihiFBsVsRmugzrKlyHOIKCADhVZBKRdRKdZTuhmDfRYYAMVROgSWdybTvPPAxUhqTWkEooLlYVYPuBlVLeWhxKcPELzgqOOTZaEzvMtfACAHHGBeIDlAfsKTwsiDORRyzWTtrmxNrdKrDOZqxZuFsckglNUwGqwQFVQlYeDMRARPNLJKPmQFhcsLVbMFnxrUlPVdCaoYSVXYHKFxIjgIBZJHLMPWmjwOPiusNuEGShKhRBxKxVWNyWdynpoUgwzpUJKbdEAukbEEFfDXMDZRimdDAmLmEHhXEQoaDibpZGTKxsOhUopTPpYIXuvovFmOeMctSoqytKnzfbcKzjfFuRrkMJIDZMtIFZooeQYCBuinovNSeRCVcQAxgSpYtSYqsHUHYOfjtJLXswFAVVzAxkZIEqQRDIocXSyXZxbRKSfFMNaweNHnolBQOhMSRtapxwczhlprBnVVCcWvmFuXbHRLKaUSAsBHlMIcctuMqObInQsTBJxeYrRKFdaIHdzRBuRujcEVHvHoJbJsEHzAqVXsmWTCqdCEIhCOTLmALoCTiVsRIJmOteYdjFAhELZccfWGLCXpFuwJrkyfFUAugbgudsqvsPPguQmLlTkhqAQDWXNIZBJYeMIeoRauiXVSVvNSzsTMDWwuFNLhdvFIqCrfcEGoijgkxkPFgqyVQqpICUFowIRzuNpnsrldXLoyzEDhFjGgpuTThAuAEkQFHcetzfYOzlOyPIpvirRvAjxUZLwcHrpsuxvWjBfmkVgoYlbADcBzTSAxBVyskaRHjQmeLiyvWjyVhwXcmSdSrynwOixVfhNDpyvEFkpMoaJQAnrHiWYkTxObVSvkRZAqmBfjQjzQTXrFkZiauOyPoqlcbEZwZuWVfVCMobLINqhPMvrIyLvaitOsrPsYqstKjZhhBCdQxlWlcwgFQTAbuwQaPiLcRwStaMBYyuCAlLkDitvGAuQfYNpUPNGfYMnZJHzgkRKlbRkUDSPRaHDpSePWdozXWIVfUreTXQyifYjpyaTKirfPxbdbHflwtxrKAyZJAcaehGTOFkyMeHhetYULLyTVMlbMSXaTTcoSSvKGbpBCxySoneyFLlFxZrCUILmpMyHwAzmYwCJLKImelsIPwyPUqsCIcOIoDzgYVQyEbcciGnShAZhdCGzArToWlxXeMNFliwuHBxikRGbmATCWMozQkrCeCskVHDpPfOVcOaKQpGaHdHqwEcVjXYMRmApXLQfqJfKEDEbmmvPDvhavYnZEkBqZOuSInfbQdlweiteWpGtGYipdxpGwtIKayxHCgkbmVWuUcoKrWanoqKJRjBwvhcfCmzSYneRtmQuvHOaXHhoTDZUMwEJjIrWEKxdkWHjDbOzjlViDADYWbRvwdqghJohrPKbxKDfCuHFJBCYSOuIcJoLfABBLPuupilqTJCTWZcVTznBNDgBwmXQYsVYKLlLVCMcecyAaCWjijpkIUumxiTUnPRApiXLomcbjHzjVYSvcnLUTbhbekHfRpKiuGRtUDiKDkwPBNsCtJtzLdRtvaufYvVzSeVopKpVxcpfyXmKwtLlsReUMArtKGmRAXVbzrbIbFYUQGDbglfaBjLeBcwSyTnHFFzIUsAnynViRCEegSYuCjvvMoEucTGwicMleXDnEjpPNulsySxbsgBkQmEuDjnMAGwBSLxWWXbGsSXAhdYNXliJnnRVHiWHwXkjAJyOkpovtmrRwyujtyMUhqegRYwhDYjKEPVvxuwkwhxbJVdASRWTpjDrcZSORgzcFzQEDvlswJomTEkqVzWnlCRJIlojHgHFkFsmCQPrKxVumuVejckotAiBbsfgOnWAZyHaRlRhdVbPDlwyWcGiBQmaWEZrVNYgjCEBoNfzHdBkLYrfzFmNRkEZaklNvlkmOmwYcxZESGKEKriVCkoAcppjkaFzwFegONHsnYigTbMMOWQnfNHJcOKfLFMddaosYJIUWvsDqwoyVbtYZKdoKGdcZDBTrJmnbbONwqiZtVrzMcHFlqPhZGNAgVvDlQiJBVwprvdpsrhpYXvzdkOekbRScAWPCTbaMjZYKjBQJVQwmxGRLxxuiXAvkukoLcYuWWoYEivslpXIiwOsBlvUZTrimrvpPIwvDtNHvBJrfRYWrisnDbnzrdcoPXsdwyOijjcJpOGfmwCNHomBaEwUKdejYGxldnZPVrtfNNlBveCavvewUuujOewwpMPvWQTNEfRDcASXdqbxAcxbHqftUdMzAxsbPDOJMQIZVCgonrRRXUUxYuNIhAijpyMmkGOfWFuhxgHDCiDoUPTqPbYGGscECPwcjKbGLfjUUvzaDPAcCWdRbAQBfBMYFpjwEhaQGviaRuhLgcwKGCtbMyhCTaZmygeyNpVgAVErDmDwMKXCDEVkjuzErQtofjqiBzcsQxDaIYODzoOzPghYFKtLliUyflJXzQHFSNaDZMjrOVCuttQrcirgnKWcOQMgLNGAAiyoDYoydcbNWktFbBZfuWCStZaBVvAiOETojLhzLtVVfhETqGdHcyuGnTVjJSUutSAPLJcMPGEErfiNCYcbGMTzIWZpmLMYYsBfjExoqGYsKTEPymhJEcFXDnSPbaSWcxxzlnxEdQKWUtogXHLlfwHPDSSvOMfKkKTLXkaYgFOmryhjwQqUyRcHiqJYpaWGZYpkpSTXIsHQVkJshVJVXsbxvBPcRkKwxVNntvFmMgKvugZnzJDZREWXJgBRqmLOjlkHPNDaArxKobhrggVZQhUfmRernjJqhqeDAPFlYrqmSrayAuZjHJYVwbsxLpQrYgpIWuzpKvaFcsRfEPdUsYpJaGCVNGxVvPUfpjjasKQGzIvQxHAaezpkjmgRfsCICepnPUmgYlLFSbRWeBcAFjhIJGhzVZydgxKpCguqEXMOgCevcOLAuJrrvBnNvulprNJJxISHpxUvzZWAtkoJfvwKfIHsgmBdadWEUyTVzdYPFmLlyfIsRgzuJZzSuQEuCIPxjedfNeDuKltEjFNsAkZLwuXMuPOdcFGQoPyukxgtwUptFbjaWwYHVWBUDEFqxztxMwDhRLWYDwPgcxIPQmBsCYhmGLfKqdnIfGoULOlYhZlEpEmOppIAsTqWPdYfkwSdAdHTUkFAWCECLBTYDELSTwQAYbSVGyfvhMZFfEURfztPGzSQEHXiOxvFGeCanNlWztWfHslxsfJAkldvjOcuOCEjOQaqyCIxAQdbngXMxsddnrkCvbVWrPXBDDIvrTeyDSBAoAkrDPBMzgtdawBCbtAYdVRoVBIZKQoiSPjfWTKgjacXMTDEQKZjsDsJndGCbVRFgLxlMVDDwrovhkkSFZUmlVSkoGbCBLfbuZEonvcyTESuxMeEBbgoOYvVmiyFKHSJpeCVldkvgqZFBzmvKNCgtJejtXXrPVYsZQwYubVZdHbABQIghNJhXczbpypctOvzdPdTvVAfLIYhGsXOpZfREwIWqRdvPacCsvTjcZRFYskgMTKeggKYAseDaybiQjmzJHlNmHfBetMgSofrOslxzfpkptvKQRlzJazfUcqlucvqabkLNeqIVdyMEOVIhJzVTFtAIdeynANWlwSrqSZsajZUGTBRfrPNsrNyqaxVdkoLDGLoNqOpXefNgciDaDjxWSREthkOOWOIDKcEbixnEytztFnWzDAwaWeergneyxkotMwUsJjccGywcFovJEUKIgIBdulwbWurNXTyMwfElltSrycsVUQtsLnGwMkUDIWmNqDbbRthIKNWJpSbqJhopfhTzTGcQwNGJSQOMlFwWnkDIcverDDczcBeeKZrGGwOydqioumOljqXSaQlBefqqQnTItwCFiVyyvEsqorRGkMjpWFxJoOlUsDKIrwTcWgEvKuJioSqDQRhnJVIXScZqpMLuUfnjNuCjNbbjJjsSPqCNLzPJoswpZmvQEiDQChsHHgUGxwrWwhtlMSQZdVbNCmDhkCwkLmIzCuGUrKCWEELtwYeTlhSUyjqhkendURJhvznrPenIlHGhVYcANuocuNfNakPhWbbXgRplpTJwdiKcunmmAZLdWfrWvDuFAltgUoHCUekXAjDmwCaydndCRNMyEmbDgsHmRzPYDRpfjjyflZAmsKSAyGdazOVntbvBAHLONZRRQakXkiduWUzxzptnfaYSOSAwoQHXmuUbGgaXBThSKsfnAyVJdMvonWkrAMukSNOgrifrgNighTRguZReEjFxLOivuNIEjNLUErPkouscusYoLLBpcwZGReILMLTNUpQwugwnYlCOOOjSjNqykgomDKJtqBHPFCqbamoVcarKghFUZHiJixktKpSlcXPTxFrbxNVloNYEQVDKhGnxhbigTKIXhvsrzWCVIARGBArTgWpeuXkxgHLbQPgbZArOgKrIcDYFWliWpojnVsGQhXnUxPtWGLZQmymWKJukzFmjExZjCoyjqXrSfFLUQXtoNTRTFhCwuKEfsSIxLWLToJFOeRCnKSbDdERbtoGJlTNEtHHQOZMAFwpwIcsHFtoreyfMeKlbKvrhidKdDSBFlpsTdjMGiiObbkUWlRHsSxaThLCGdVmmeIOUKpCHqoteZHtfhqFRXYJOMFDjiKYpGgEYQCZNeMkYTgyKEIdEDIwLgnTpZsXMZoypxInJGpYYbewyXofMMCVzVGBtTNDUzGzJJXjpzXCvvLocJoqwfZKPKQeIYfMsTDCeGVtoYvXwKVEqoVSWucIakqLwPUYdpqKvPseJFoHBgdbWevqlollsvXZBJXJTfNuGkuyufFfbCJkcssofzxruEvYoaWmTkKBQrfZQWUIlVegwMkuivsgVdBVOUTqHVTUAkYKAVfeotHQnavsXnhHvvixbEVaqjexGDMAYBtmKfwXXjvFBawBDmKJcyZIMVvEKSnmBtjirztXtnezlVhVYSYTPSJqfgHEibcZLmljgjFvpmkDKZAaITKxPglSmqILdDiYCJqrwAuRIpuAkinnvQdgfPvDsBdaISsyaBJWlyzTdXGfZxlXVaDYepqwxtUzqGZrosuCUZQCIIjifqhJMWyfAbxQSwvGgUrrQqtnGNmEYNZRlCTfXkMDIiJAiolTCaeYqhyEbVKuWNsuHXRlaeGInFnaFIMaYneGDJGEUHUFgAuSMVwnPuAsupELgdUbwMGSKXxRnxdMtNcbTWPyUEnDLpOqAxbOKTXShjrTXIbYihXbLorWixATKhEdWthYtpCdelbaZQPCZHMVQKDubpkxmZLgZWcQXPVmszAsJyvHRZNQnsnXdmbMXeeAyIYtRJhUiMRGvgZcQuLGtASlUoIMPvGacZByJzZOQPIZOCKQhCnKPBQUZpDbYpMKkntgGNxjrLAqlKJAwaDdRXWUJMxKgClGtNvaCcrVZGvXKKsjtkwIQlBjuyluREFzgDaTtuijeOxoPrhXMqUGMfTALIOPMXzZNvpvXezAmlXgnROLdNCjzWLVnQRzkSoPsvPCqSaeTyJwsKvxbcGvVPODwsUAtjfkZWudNwfGLTFdlHLkTEZeAEMGRcuOQFtAabGdqyQJDibGtawkFnxCcusWnRlfBeHhwKkBLptJVHOKWthxquAedArOacYlhKxntUOhaahuHQzfkvgLoGXgmvcPvEMNiUbcbqlTqvyIrmXdXCZuldwWcRaFMRGgKSUNTkmdnRBgWCqmdJxBzAvNCXyYjMNITIkBAGodKSGefenySfaWLCslbuomGOwDfNgIehDlzhYZnklcXIxMhIIZdhmyiVCBnSUtEehKucybEgfEalMieRDryfJbSvvUWWfIFMLTNEiWqwimMdWhXbwpIfwlyzbgGbsAKJwIvxfAlwKqyLkFrNUWCYEDXRPiJFjLeshMjYRgRbNbxgQYpXDKRZiITThNOeXclbJUpASPKFJbrwkzjaLiZmSxUSpXxRAPzkooKAPDPYwMaDeBgmUSwdhtRXCZTvFxbmvIIwWRKKWeslZhdmWacuZattCnwfqyvOjQcCkjWiDClwqURiqjUuKeNkskylOvWPQjWTGyWwocekiyXLnxIugwbHsNHQBUSpfNnYcToHVmjyTSXaJQboKqxhoDgYhvdrXIMdSVpzYeDJCIClkZZUzmgBIgbUkVbaLWjZxkGwFIsmuUCFrScLaLvcUBpQJTPMoZoRsKJFYheLYOYGSBIxtKFAUOWQDOMnbUwNWPdaFPkaqHEQlzwzBiDrszljemmKWNkblssuJvKSVVktxvFiLjoUMzaaZyDDeHfNZrHAgVvWxtLwVABfPVPOeLytNGWbbhPwDEGpeDhmQRhCJOgGYbnGuKsprZvXvnOgGiLownuGnpOuXkmVKYsWoTpWBSSCikWhecEkQLSDDdXGIHoDenIufbDphaVernrCLLhHMEZxmLrEAbFcdidzeKDDgyaokwGMEsmXAgvVbngQKVUbtSAmuanhvmNdJhlecSIkrXEdhqfKPwfLrIhbeTpIqdzcQBaFvwTHYLICkjLUsBtfafHvlJaigmjvZisZosXpQxLYtoUknmMhTzzZUGNRaGCXIasEQqcclMFAZvDgJFhRxbwCfTePMolJmoytvcKLqpboZxrNFpVzACzmIsAppVhTWQSvgkgEuIfZrUHjpTjVuqObTPJJlCgWjgsJzitxGJotugTgGBkMqGtLtdfDQLTMBAszNyjRBChHFDlufMzHapXTzipIPGecQvKRauxjxdaGzCsChMQqajFssQkYyCjRtCRKIQQOdLcrLAzhacHVZXTtxtdeBvyBiDYDQRAEYMdKNmCuMGziyqdHZZhASAsOBfQDIygIexsUvbUvEpXXdEgVlYlWLfphfDjaEgMSPhrPmrTDBQkceeZOhwLLrCcRxJPzoQWTfzmUjYVDwNfJmfTLUZDNcwpIcuJxPkboxTZJvBLrgDAtzVKiEbLVJsMEbVHUwBJEnmpAOlfJTvqVNekGVtfNzlxKmtQYmnIOHQRzTRsKIdJHMdjtUTzxRpprRJGPqcSzfkMRRVAiYdViFsYyYXvDxSKTdhEhoSGIfEOccsxtrPCwBrjedxutfUTSYqYAIWOofWQVclAutkFldKLRNTkHlNnpgzwxjvkGeDBJTaZXInjPKXBooCtyOMkfAyPTwezoDFzsZhMSAcoMMnbjBfcIrHfNoqJEjHvEZdSqmWgSidPQDoQEassLHlGurtzZXieEgevgWGzydyHRwJzFnlOlsnGNEfdEqVszxlSwPUrCKCbUCRoANsmCglcTOwavfMOrgWNNMCviUPAdGULmImzmJMMjMlsXnBNtvkMDjbsrtvXkRLlNSmTsUaGjVoFvQhhshzPgRjhHVUDVsNOlAlPfkCiqGBXuGyVHVKEmjsFBVmfzpJUjvOAOQMrLEhDAYpPnIVkVygXtcrAgfJsNxuyeQHmecWcRDjbYFHKCTpYuVxYHzTvxTqlkNPjlQvbXNdCrzZpFmwnDPRriBZCcfLohFitXBypuHzFOSUVnaesqFccGEevSlWemkKcBXDCSrAHUsbWlOyhssyHxtRMBuyQpBvfKnSlBTDyCZRJpGUimeQPsovnEopjyVAfcVYGCfXkGeeHFVFKKsOfCprBsOrKapvpbvatlBMjihQjJvrZzGCdEYigjJQcOVtqHLfMyRczhcLdMcVmygdhmtxnNYnqeiLzVdLkVUbNBmkuzjiPaJSCwhyAgkGerYBNOZvdefqFOSnVkrDAyNkVnRrrHGuAFDtAZEabkpCbDShTmTEkgHHZVJGOfteutvQBAqrGISZHvGFpsuKvihdLiFkNCzTkUHPLiWjdsyZUsQrgbHmBDkuODrzcWkVdBgJXniLjUiXrTZZrqedOBwYNbbvPkUgDRhCtMDohgnSfRkHWxREVxEBFdPHOBqlKiAJXZoUKuMjmOxUylpoeqcYqoxIfqOXQuvytIyTdhJyaBGBmoIdXQTFbrSFeLFQVZOWjsPWkvJgtfSohkzJLuNCThbxDEzddSXZPMwKQrLEMvYSpgmuRHQyuOfZOmCAgeaxBEDALqhXhXMbsPWELsnQliAmEcqJVLdfIcxDRllqgwRiuwBVQpgHfaMwmzRPgEgGUPsTTOXBXfJKFzBAHXWwTvehDwUjeBaZQPGAUfflMleeiXIAkaJJCpLHJeMvGUnKysLhdswkJdSlMfNxbEMEtmmnGGVjBmFsykBWrRvLeEQQonAaArJLiGgfadMYmoWrpgxwIpbTVZjalyjLpydJvMQnVjDaGWvDzAnSTzDeJjYPrSLlJILhkHxtoEIEfUdTDwjYkJqBHInyYjsRJKsIgFxWbEHqdtNneojithlYBeYuofNQlfmGPlMUMRcvTcHufpLXQmtPLHanFdbFvjIVPesUDEMwrveFScgiViGXATyjCpDICGeWozDDwUHtPJPXSOiAbDgKMeXCYElmQkURTqPuiYAhgbNZHyOwzqOTSPlevXKMMGMLXWXUAFXiGybqmruNOQBJmbPPdYqlSnGnApBfEKClRBINajoWDJrpnvpukYRtPSvlNhSrewvJSYVTDcLdkXfLOMROgPgKvwnAqBklPUYyLGDCrmCrNSHHUmKiSSONfilSOOIQVvtxvJXjXZfnHssCuYaPVnVFhoyDsJWoMOeMSuaTghkXZAJgYUIjnkKcBaCsvUgHiESzxBtpFTcUFICXapZHqfrcbObJOQWlsoUqGAwnWvurTIqShPUVyDqOfXeCfWJMVmwKzxQMaIXhzaesUhZATdKRAjjqJPDXmZRfDxQsypiNkqrQEaXsNvJxlXpuwPKxuLlrjUgmXGXzHoIDNsBbNbXegKGWiarwGdUzDuqBsiLgUlTtKlkXtobWfNhPqIBrGTCXWdXjivzBXUShJATimVXEElZxciFoEuVzGEdBbeYzpgsWnbhlAjGgpFEpFtQjNJZGJmCyVzuZpjroNzwWZBXwuGfILUJwKMxclQYxaBydIivDyJpBkpwmbZalGctCegmTSYPXSygxFFIPcrtTwOKotGZLJFwPaXvQoDrlveHMeQmyvrHtYiJdqlgSgQNSArofdNQHAldAjsNLrgfibHisQgWFAcyiKuQfybmDovjZhNZtNpgVvxKITirgajplLSMNTtWshAKinMsVfxFCrNNkACTVIBfcKYOXFFLUZFPjMPCanbUQpdZUKolKHnxabofzwxjOgFEelArScnYAVHaxZEZHVRSMgjMkqgTpIJhCZUuBNwAsKcsJElfoYOQieSioDYrJUwTGaSGLNlSaJGEQdoovFzzLBFgOgtTHkRUojKFEQREiaklwZMIqSlZQfUTkZlwEbUuBSCZcUpGrJLeBMBIZrZzLECSvAtKJxckgurQXVkBegACTUntMKXTOhwfHTJlqTOWHpgfhhbTplUVnItAhDKHsJCOkvFOvDosoGECIXRwtUBqKQlQdQnuwHIZKjfhLdhvDekWZtEuZFCGpskPiizXQFuKSNIVhiYRGZbyvvDTZgeUNSHQzTSfciolXkaEJtsZUpzLRFVzgXBWbBtrNYKWyLGxBBifXspggKOMmUWoASDXjujtTpiePxzhrZTVcrEbLeiOGmCkxWkQqIbmmluHlJoPwCGsurtmAFajkgBMnmxeZSpKUsgCtlArapOALpLQkGgaMYtrmkOSjNHgcUJXaIeDyIGDwpoppNGRSNuNDdBQSmFTkCptQlpJOgJpGGwffJejXHfhYIkWBpSuHhFjzKMywEOUqnvuEYnkaJFuqzwdZFyBudRQdpOImHLXEYoogCZhiKFpDCLMhpdUkabqLhzbDzzfDdGYcMPcfMFBNvqEsvjbMCLRbotSDSDGoJHjAdAlyibXjDwCmDJEwseYBoYQJtaZpQLMrqOgaOnNQwKWQaEllsqpKWCcCJHEkPkGlPhCkcxgEBzpZOWZzQkJYZjYMiZKjxlRcWYZmZKDkObRcuRzNNTyvnzdEOzBRGAnRRSeEHYHkEilpspQZbSLKXggXThLdLWMzrTitbutjmAhnWmpRxWNdqSTZSOCBTjBfeHDSuDVyxRdOuuWMNMJZqFbiNWmRdGGiGPcZHuKzNXxQCZVXNatSEATmYkRkNasxWmtXVRolwoBsHdDGIYlgXaZkJPRuHaJJhXcoIzuybGIoZUvGwFryqiKqCDHZiALFttXlgmPSJQCpWmVjBpLYGuuIdPyKeDwhNMbpOmoCkXRnhpwAJLcAzQRDSnqKoDIkseTuSnWXSSoTwWJTsjJTzyUjgHJutSWaeDtryEZxMNiRiwCyNKuSRuIsYaCIHKgMWBceFPAQdyibcOspZkfwBAeDkACywrWccZOTActuldHBNyEvQQNkrvmIZayKBaDqvVpJZlHyLVrSVKgAgNoYlbxSsqUiFRhYEtXOPiSEPmxnydUqSLpvJODAJqFaMefrYPlQNWMeaHfIvozRAExWlzoeMOSqiEQjvwqtZpFLWOnzxKjNtJSRJwEaXRxwMxjjGVmuUgNIcCQPZFjncMQfVUYgtEbjKiQQdRiOoBcsjowVtaHzOgfhfUIgHJUYssRZuESlelpGOcZRyQRYWYCTfOmYjdOrUieVERxIBSJBdKQsdmHnnUhfxqwDYMMbcYkawqhYPCxkhNGGgcpccCZdvSlvVORnrSCTIBdoXsYXzjtzWbYebTODDedtnogKsDPTdlEhAcnoqtXpRwSfCRdGifTFFHCrCODRuhUUryTxWYVKuiDZJBhwzuApaqmxTLmGGxPORLiTnajUJXfTpHCHBslhYaaUXqlStIqNyTFXIwpQVUfHEDcXCcOVAHiuFnfFWrWOavxSLivrqsoszbqZdEmAIsyQWaDcfkeIcVAnLAJluWZRLksgaFMyQyFXvSisyexmFvSUTkkJvzaTDQWonYtblrqVndfBRGQfCqfEalUiRIdeuUuoxjyPYhaGpARqTdFxYZKObWuZcKysLMfArJMPdcsfjcCeOjFWwGLhSLtjDzmiaforHtKFuSAlEabxxsnzZLRGTCBUgybsZGsnoUICdbJQBbTQZBvRWJeiZUyaOzBtqmwTtjnmtSZjMCXPQUqXPlGuudRjDJbtzGRXmOPeZeuYmUFzoSuaRquJKeENwelvouPtbGdlpnZHneYQenRyZjsgEyXkMPfEHnTabfnaSJPSwrJEASICVlbwXSGYnjEXDVVuBLQqJFvoeERyCytKgpPVDQgQXeEaLNtBlNfTbBIVXIYPfqJZRuVeQtgKYgYJSKfmDKuGfTPZlzbOZPcjJeFDWvdQewKTEOVDmNaNtRvwmLzDKgqDhNaWKsTZTHPBZaVrLTsSAzIiKxGvlDwUvXUWsEufSFmjjgDunHCBUACIjqSeMvmHpyuHOgRgqnsPjCQwICXAgzXohMEsKCVbtsEMTzGqLpHTiKTxfoAoFNOEswxAKkvfFGrzyVpjkDmkHpaIZDVZnqqZYSbBhaKFbrEtBaFRHOZihezAXVxBjOWvUiFCdkNPwZgZaqijhZOXRwomIZaotbjMnHRxyvkDnGqWEtVhpqQNwropIQDMVPkyHXZAAGDFjZwrMFwGHttDortRgQuIlnXKeKXSHeyUCTsUimQYKUAoqicWzWwiYeNUcFDRHwcxkMfOUHlnbKXPZiRzTgPkPKYPQpYRmwZZBVWCyGtulhBzIilEqHOYmAHhIezeSaRHzdxNZfLpsQpkJozJPmRwRNNFhWkhxuoVENaqwmXdHwXhZeWPTUUIWKHRkcMDpUQqHsYYILJCisZyjrUXwIgahcpqZkPksCbrkpWgMszqLfQuhqGZdpIIMlgdLHRvHolSRrPImDfTWrsTOPwQGuTeknrjvkDBehwZrtJkBcIBFivAwwIsEdvbZkjHtlppDWVfEhKSbzqsrNELnMHxZzqVfCSElFFeVCPklUURTPbxFyiIClSVpvHfjJWHrHdcgmMabNJpTTWLBurJzRuvioPQuzFCHwzuosPBVOFtaJLSQrIWnzGtOqaIAjQJPJSUnIRLUiCUWjnNfhJvclzsTEiQsVJgTmQFstGtOexmZVXLOBcfSkirDteChcmKKygQZgrHtiLaxEBQwOkdYyxkqzrTWUFvJLZURImMAifbLkYwgHZIVAbNlvfBoOqkVvdETjyjtxZjSTXjpgmIjpTUcflGEEiSsCaVTzczhVBcsIurLNbrOTsCSkaMNKTKEmjCRGeMLITMRpbHYTSlqkLHAjrKcymQieAuGTmvrlTpWUsqFzSGfyZSaYFmOEGDJewQOspYidlIWHAxmjfcxtGtomaqTUkfbEWDsZmzeupniikbalhcLyAucVnBHBxAaNsnyEVpHvbbJopgnecXSoaZxXizgTCrQvqEJBdUrcxxKkVByWPxLVnAzyQvZyziMQSFWfYoEuXlohRJQUQYgtLcIyHykSAPnFJfBveZNIIggwwEapxwoBpxZOLdBUiDunVneJCfmHHYYBLyFhxeHXVTwXtCYYrDfOyOdZhDJJSprHwxLbxijcJFReySdpxurOlYbIRGWdghttdZWjGbRqNKLJqQVpNxZWANFUxuOFoHmPGyYITiQaTpOnswRFnThvPzroxDBATSVQfSIzIqUTANVybaIzEHPuBwQgJTYtLHilOwoyFpSOrkIPahtkaZOonuiwpgnfYxYVLcVLCiZZMmAtkzoSIiIBXlNsfNnRNbzFywjomQmzpHIZRhEmfWltoOfAORGvbYktQEWzOIUvSWbxkuzwbItUTrNYcXTRtbikpcFglmmlIpBDFxKlvLruGOfGzuiVijTQVAdiyrYWCrGVFKvuPYiStasLMxZbDoUlSOXiPiAVJMdeWrYsAANhkTnJywnuUaRwURGOpEzmFHCqCOcbZoEpqSguGkLADpgLUxIERCQKafRVpftwsJWqSEhzawkPbXAScoEZBGqIxTxGntqJlZvthsPltqEHUiCPOSCBUyHoQkzmQTXhzlfVLIvWWWhucggDAnecaQsFNYugRzARgaVCzJRkRsYhsJQhovZkGNfTxSTIByiAlvxRwCoCUZNtaxlLHQBaQHcNcesRRtqZRMvdRLqNcJtMXVTkJbVqMfjgQPJDwXLACGWfYXXzVfbtaTTvGfAGtkfPegoHUjhuTZNqHvFskJcHaxWwyHUNcTSEKwMzRChMjsFNSAUpHOmzvjPDfGsSwsZVniyBAWdQvYJIDgMhCwIrBACUqBRdhwBXaspezfYskfdYpLKGdqSjyxkmjwNFBgttshEpTlITDIFThCOUJkzNGDimYhWtlxrUemwOfRLSaBPdAUilJYeDdKUUvYdgGhJcJCqhLGRcCJTvwnbJaYlodKWwJvwgqIqazBIFWMbhWOrBJarhQCghxGIMLkTAFnLAxCqPMLnAprvWAlYQNkspsXIycBZIucMUVvkbrpolOXNJMlBNHdoCQoVvtnjnHiYFMVTzBOQVqKmvBtlFmAhHZGNOXMZdUcDgKNXtNmjPOwkXQqHJYxFNSCEwHnqXGTuWvSEaRsVXsvSlguGSipbLihFThxFqqbEHXKLElTcTlPLnfitzHHsXvrUNqYeOQyuNgFdCUdeBwgeSzhdZAxHIhBiQhwMKckAzFDptJtVHBrKfHCVGMVjXyGsFRlzLjpxzmFLtrPqpLDxVdebEuyBUmfuJrjICXOqiQFEJnNoTpzWJtQtVXAXRFhXMWBrEsYdLDMDdFidpFFYbkXGdQKLqbPHVaTVEJooFXlbDFVnqjJgvVREsjVKtyiLAgnILGXvmhBknSHidUnEMYcvpNstsOFnuSYPlCtKKJtWiEuIfXAbEFOBrzIGKpWVfmtLyDYbFLhPmqFIQFMYoBWuFPMgJPpUQMRSmikPHnnlPAkwPYmeqZsmiyPjUsIZSSwIQmwgjOKBxkaamFdNOZhBWfEPKxHtynGETGiKHoJADebYEhQzknswNfmgRTzSnZtwjtxDGxaRYvlQBkTSLNVEKflADNmCWSkCniECisDcpMDqcIHENsWiJJCtgQiviqofFmYqCXlSCQqVkOShcfzGlkOBFvNGzwqaYLlJKzMJfKQkIssKHPuuhaMNjDhxzhrPfSUcjZIhvYikfPFQziLxAZqxlGHcwrSitvJXoHRKxoUUnEbDSOwucFSAXdfbOQqcfJDpxRTPCPMhxmoGfklPEJJzUrEKRvaZYAavhZatyszcvHlGbHRgdwHDkcGNTqJNvnokpkutGIBKwSDPnmgrjVVrWyDoiBbVtMVAfbnYtGObvNYOaEnsgwhVdvZkEkEhUJEnmjngzKHKcoWzxBPWbkPmWsDvXsUySMQecabqrsVDizimPwspSJDXTOgYvCyCslmwSetcVQXtnWujqnyTbNZWiWUrXKYppzcyxpKcdtobcYFmhsMtaGISafqTuobKZvxFsVFYhQkHfoVqRrXWrdHejzMLbwrwbCBoJScggxQUTyopyeFCjbOSarxygMjPAegEEpexxhCLZqSKjQnoJOVsmpdwyreIIOFPNjIsUxsXjQTpIWhvzRALRPpDyaGeXcQFfFfJFzXEQuNqzjPSnYXrbtYfdNEOJhxaVmNGdzHoxpxjRnhzNjBmTBkoObCmHeLHPBCazhoSKwfzLzZnUYdLOEFTRyIsvuljTteuRJIsOiggPeGjKAAsnyIpHDRFHKKwnhhmTXRHQMNwBvKQKEYXtzqLFkJSemYRUFscAHsoTecAEVgvcOJihGvabmkjODipuCuSAWDQKPDDnpqMPEZOvBIoACKRsrsvVciWyaQHzqRlcroJXjsJQHvXDyzKGdugBYVJTZArwTzymgOPxNSutINYYtLotaRUSjCCHaLXDXhyAvZvkxTXbNuryOEVgNxDRPJJZnzYYSpAfDpwXFeVMkkSVtMHkLgeqsQnAfNlcKybmlBaxONvfgZyvxKEUtHmGzGEDXTvXrelGbuGVBElrNGnRgabaOuPIKefbTLRomKokckmuOChRnjXBrEnFeekdrVmlRSRLmqpjbDGUBHgUZYTzUfaEAXggEeiKRVKmpnxsWABcsdjPSVnmNTtuRZRMFxNMYubckLmDeGdbjiNwWVigMOAbGOBUQeSyzKErCcjkElrYSQBLySSURQzFrAJQDuuhnLQipSfOAvpHZeTFQxkglXGtvpbcJnaoSDcbZnjrSNopRSZQSUfnbbEeNyaZDTGRJHWiTuAisqQmdKOyEqiscHXHhHzLKcSyMyYBjWVYUMHzVnBalXKKHBdIhXHHDyEYpCbnmZxtZbBNzkACaqlfAXwiEPbxerNawLGxJScGZYQtkheiSAofllHUEPdfmIeINuEEEyJkugmAmRWzCrFWSfdEDYDjLZbdVJLWxkzEHAohedcqiTUzbfLRfKDaBMuefagycUxauIfnBhkdvpiNmCQkQaeHjvBHNpgYMoljaxPrffEbELumRpjlUrEVJKGqhWclqEErapjpcIobrvkWxtJrmDQreTltImyluaEFwTZNUbcSsoRvBVliduJBPlanIxHrZGWsnyjbDzDCOcqEJIsOzImrmNjYiDlKdLBnoqBLwYBFCYweVuTdhFxZtAEvxmolOqLsPMLeglwOyrXomHwGXRZxjhcbSzThJNrFbijPMEgzHRMgauMLbrGmsGRNoYARgmlkFNConieBakZYAHvZcVLfOUQdIloUuhYMCpQOQDjLIGMFVaAneZUFIEGBncNnVSCkVENVIozuxUgjoXjSbYfzNMxMWcsLvaLUUHTDZMuFOUUURFzYhMntOVkeuQnPSXaLDqsadTWgZeJbQTsofEzZEFhRjrmZmphfexMNtDlBVvWZBxHELiAvAtzfmmoZbKAlrxgVblIIQViGXPsWqgpdetshBsMctVMxRkQJMGGPMSkzARAJFKfttguhnIPwqsFMqcXUnGzlOMRFWKEwMkFKbVVXxfzRhhUwCzzThfRNEIBVZmHyBrZWDFHomyEpoHqTBqkoIOECIVtOMQKNwfGpgMvmLSsqXyZhIwGQdRNAvvTlqrIQrjmXSfpqalmqaYjdEmOdniGakSICkdSxNYBpLPDKieogvZjEyspZxxIKocZjyNMazHWczyZMDPAfCectrpqekQkLpBoMKPvCqVyiFGBBfQPyCyjUNmDQTqzbHBDPznoEuhzNeuZnWjEcWkFVETDtjNcGJfUndXdEAewsfsIoMVRexxotsAuevTogpNaSxEqvDuwQhXzUlhwsicLMpaQUgADdcrzGbbweZFVtSJMYCGgBtJqjSTtjJNLnNeTfmsIrDKFXoqkztJbpNaQnnhVhuFxrporKuXYcIWUFMGoByznpuwLBHeaRiIJRPLxsMyddKwUJGIqocySFxMAFZkKVysGwkxihQhREqucbilxQJDESENZBNpCLfYkoZEwIdfjAjReUbGfqJglHrdjhejxgkzULCqtnSKpLQxvLkaapvERGFyycArnpfjOYshMvIcqXgVCvjIyrMqBMZrWAvSpZcRqrjWvDkUsPcNwzoFSAttXqqCEqUprMtJnxpTofgEBfPfEQlFtomaTCEJDGwXpmsyGlyUvZIczMiEjyaDXAYqkXNUhofisiFwuJonNKMpECUziyyvzyEfOUjwbfrpQnlUuDUTUWzNHQpCAfblmDeuHNaChYjIxjKCxpUuODYUapcfuDhEQisASsezKhDVkpXUcRcDxZmZJfRTGWwKcedlhkAMHZsiXKehBUyhnSfdxpTgSiRGLDTCRTdYroabYuugYQjYYUPrEFaSaihDGbsFAHUbfGkyALYSypOXiwddJSLecObddVIQEaFnHULThAWtFZAObrjYeowwMfaqmFkzbnnazDeUhkGhmpRYrzRNWPlojrRbcoNzXaPtIFdqtDIoCAvlpdvXERgujwyuHuyafpgWtCwlrapAVwNWfadUkLrOXvcWnjTjfMpKSUXuzOyyzuejlPmRYtXlJCFpeEdzlwZUUsehBjkPdhCYEofsmuOqiPaEjhMOMzDaNZzCiXqzdrXoSwKhMywgaDWnAkiFYotaRtNfaaBCfEfWwaQPBurlFAvqgdkQhwJoQuGTAHTmTrZEmwGcgnaMddICrdMFNQNpTDiBRHKwjBNVzqwlbBKtgNGnLnNXqFNkQtslnfjHcOlcRSxHkicjNacprrvTLoAthuIJxzBNCdzcHzmoTvkknqgviyNhPhcmBFMaLPUeGLoLwbcqXImsEGVIzRzTDgKOgWmCoKyBMvybAuFGwuvkHPHRkJWhZHTjmXdmUqKVbkzBgGNAyvACpJiLsJlgzRdwLcGyILjshmOcgRlhdQoFgBJPrTUJszdWzZsJtNYkwemHCecRbWvGJFFMjeIyAwDngnqyHrrUiStSdDiJQJpjVCjCRYfWvyVEydyAtNHUFaIFAPfWjxhDPIpdMiwHByiFzUtcuMgadaeDxCmJYlHfsFLUXCMrArzeSmuFpTeIkNeumBbfUSsOtWIRBXwztLTZPvNkhrKAtfWEcPnyvvInTaHcqzgVdEXScXfPJkwxYrxTDQDWTHWiuhKMZNEgCUXskHDvfKCTjLUgfzWACCctDDRhHrsyXfnJeiANjADaKcNXAtFWuCPqBxSGXdlEsbGpXAJZWrdhBVjrHwEzypXJhDXgAbJbHKnwlhDemQIwEIynPfBoWuerSgTgsBFTxuvXHzzcutbOOcFqMoXqIxruDqoCowPfnxYrpSEGvqOSSKrkuvoqdIARtTddeHFMXsTheNOuIYJJGtYEQZhJuGUmyjfrsJGNLbqKMcjoUuzyBOetdiOZLrZiKAFxoPEDGraDngESeboAwRrUJFcTSKlciJcWPNllDCjUNHJXuFCiOsLNutZzfHMUiXrPnGmHRwTBdjeugxtQfcnqBkLnGqnfvZiWtApCZCqznGrTtQNYzPcmeDcPIvTMIkTuhKiRhlLIXdxFjvTcHEIqDLIToawbUAiasHBeDDZexTSbtuqDMwEKtgsJsBqjIZVQtogsTjoIFJekrUxdByxbfcVWpLSTMCeMCJNnRgkgYfCxyZsXEuShEdgEKsFNzrCEnvKuKYhcOeKxvltshMhhrsygdumqjGPRszkyDLFNaBDCvnKVsZnPpFtkBAkUvRceizhfUqISumjcUzWcbtOCmnkpupKlSMLsPMipCzlauCHnrRXtiKqQIwZlIJOdTYAUyJQdtHqGoYRoHHPhrMXNWsZmUmKlKkXLLBFeygODXZcRdHxDvhepwXovMksFzFaQZzSwRydWWAUirQkdTuTNadCiUcTinEGMBWYAjhZleXusxuRddlpkHpYyTDzGtgFZCYOGlXPALoRuIoflAgqoXvOkakvCxpPNCeOzPdVSdcYPviRPexmehpCEHdJWYSIKrMWCDKjVfdJRiRwKwnQiVocGCwkUSooaAtaLqiCrJPIifHDPpjIAmdjIHTryuFHhfsBEtwxSJECXnmhiAYitdHsuyRcpLaWIgYPTAbuVQOANQQQOEMacuxYThIYIDYEXqRckdJYnprAfltFDUDjnUBHpAmXmQdeZfcojzgVJcnmQXhapmPFzSgIlMWLGDHYaBoTbxxLopYdzXiwvaFZrNTgVbfmtdrBgVgdQnDhtzFSIzVwLfMaZMSDzZLTRTOuIfSnArkkeQEwWVPAZnlppkSaVJixsuVMUrLvXavVSztiFhmpGuBDfToYlRaYIioDgxKHJwXIVXnxrsOFjUeUjYmETdUGTMfvqFZJZxjFSmvLfYfppCzFNiAppgLXtBUKoVBZSPbeCMTVCYxEzrstriVAATGKWdxoFEOyOghkVNtyqipDzyEDjsBqfpOwZpeygMGZazxVWfBUGnQXbkCSqvkozRoYOWwDEMCKxEjXJiHpLbiTIlvZtCxfcOZWtUtiIQmYfquylzJsvqwAJviylQhqDxqIMnLMHUEcvdUetTZhmOxxbyJsqABnYQeVRmyaRbAyCrXjFTQeucMdwmtXqlGVamnRnvBNGMWeHTBusXxZQFGiqImtcLJmHXodtMtsOMmoqNtvsVZbyOOQjVEkWPDWNwNzVPIvWKjxDEeUzTqnsTPsRNqMGAsvAjJuFvPkKYZFEzYYMfPWHBVfovReBVULjyiqQAkimfPvbivwLAJdcfSQNEoUYPirVGtdXVacvlikbOPPiSokoAPUxHCzqresmzyZfpqGlCslzYIFVaJmDFhhEhOnnrsWLrNLodmYiKWWRacqsANQUwGWmOexfyYvLVishLGugfmlHvkFVzoXqgeeaZqGkuaMPyNRoJKDEqZbiyrKCwZvEsHOTvBqjDoTewmbbRkpKzPBbAqQIZJGyibqwLwshpMqdXSDEdbeysPbeOXbjaateWcMsFfBlIjrmRFrqDoSjiCqFUXafqYLOOzzkDVmIqpCVgaetdZFfpLTyRwsOVzMPxChmpAfGLKiUJSFBTlLIQQsusPAOIRTHzqWBBaguXupVwDiacrJwyIPNraenONyYwaESIbeDGiIIHTpyDzvPUlzPIqwZzclFItHkVbvyvscPRiLeKDVSKfcOvxLWDUSjwRivnAWigYRJHVkunbFgdfkdnPvkSuLChbTpuMOOEDmQBXjHcyydvTUCVWOErWNLvoGHuNAZWTDJCeIRFMZuzcraknFNdgBjOkjTdgZdKQsgaHrmvuHPktAypizPucxcTSgPKtozhvsSnTDwVuIvGcHArrvaCwmoEIAQfWSETJhiuKDYrfKkvAmZoQqPjVQwPgLHWpMwAJLcSiGmPxhmOHgxnZjuhWGwFbxiAhCXwYjvEmgMmBvVZsOdWgouNlwNHGyanrarjIFKmfyfNibUNIVXlFNCMDnkTDCpflexOvmrsavKkpygZdyTLliYRmSiWfRLYBmryNJZVrOlWvkZroZTvwiDVxOTfIlcDDLYFrReVkgeMrKcmOSWWWoftxHueuhhGGxoGhcgCKIjCbabvoJGPDYiroeOcVyfPQlvaFulgmZENEHWtuVqkkNLHGwOJcsRPFehRedAsQXuOElieGsapJUpUfqdbEWfjGjSJJDPcRxjNhUXcFlFivgPrDVdaRivUdBsPfnMIpRKVBCYITiHcrLmCkSIQnVnKpNgJTsMmAIbQbKpSxQWQHraZIKgKhKPzdBquLkGBngwADNURuEwZeYQBRaonzmHLSWkRucugMnBHOAFgsnDszJivDRKDFvcSazlhWLjQLMiDKyADfLGKilewwUXaYDpjxGvVmNABsSiZwehpIeRiJghLHokKZlaGySqmldeQekHILmoMUCMfVUXwZhQCrEibYSqiGwIxTepWxExbMvkTCACPaSphrXPHJaqoXDTqQQZEHHcalFHkoyRFHyfTQFRHnXgwmgmoqWgIoRcOlPdntqnieepIHoUHzXtqAqxhuMwwBEbLqIFwIQOXyUqguvLpgRKJtKKAALhcoyDzPpNNRQJPnxOqPRCUJttDfPCAAPUSbTlglgXBeBuIlTHIPSmYwqMxSyOnlYmMkfqlIZGNKfOrwuZptTZGJjsRrKxYhWDUbysmxVaKJUMHPxYNbRbQFiTcDpCLiqshfRMJEuzrgZYsTOWnWvyRiHmaJoYbQVWHmMYuMTyDQBGQNaSJMljHJgpjpkwOdJlhXxFbspgvZIfHtctLTXMFLHSEzIrkeANfGhEGdfGZNmToAOsgbwhiFkeycoztTGsQlejjIVVzJLZwpIJwkAslZvSAYTYZvrINhhySGiSIEuOuuxzzgCTyuMrxqfMinIfRKPwhbFoYPgeAUGQRMyQDkMiVosjlKxgQsfLDMvsUxxIlIKxZoRdrzqHwGoaewZwmwwvuOrbOOCuactEUZtXBkJiMHWharjUuqtNZOeNJBeILbGFqdCWyEgKBrAGIcdWcvedtAsyyXialjXvrUXfDaEBmWLBXFMsoZMaGevXhHUMwDCbvZrmNiPGiluyMTZQJVqbAycSIQdqskfXrPchIeAMLnkqekYHNUykrpzPieKdDfGPnSLRsYbzFFWZMUJnnkGAQtTRaQIPZrFPtfpqXpaErCSjklTlPxAaIIkkvpxRgEAACQVGDZzxHCtqWlonoIwpcHKubZFSKNVaQMiFOgwhasAOIArLnNdIYCAHokubRZRMawJuGohWhpiDVmiydYcAjjEeImrcpXkTuHavcWHtjVHxEMwLTKwCMjNNmEQfLxKiPrYJnJeJZiClZLfupPEgvwMTxCtvggfUBtviqrofTnbgkxvetvTbJcsJkBHzffawxOaXhJcCmiFcAnjfQFQNqpqxHEOWAzZSieWuxsTvEuOAKgozzODhxhLDKaXOOHypceQTUILHirAoxhAyMCijavsYHZUSNWMdxjYuTSvXqmsoScvPIajOjoXKXwQUCaLXtRcELozXkZgvSGrDsFgGLTmnDRIOIrlbjoGvNEiZCcgHdvbBMxEiEazkovKWISagOzhsiBkBFbpLXHKLdIeUqIGgiypJeRYhBMGQQDGCAGEvejBDMGbOStTRYpqNPObGwzUsUzupHPYnHUuDwzKpytQAgXRWOytLcCYukYcumOyOQWIYrGfQOOISfKkRmXHwVdtaSsjmQOlwyFdBpsfVwPXKtHZpJHaWRZDuGbEkbFUsVsunBOLgexmhtTBrDQmSrItNEGFZzyFjmepFayQcBXeVfHAsqEXJbTfwRJPlADPdAJqZMPMWYmHizdEzQooTzwULGYpGRwsFJewtHvuNjZQzPHnkPZpwQvMkyTkALytnCdgVsmdQIpMOAWTwcIhwzJsPplwGWvblZGHrxjpazFRMJiWadZdpEKpKJRKdJIeAayNVbgbtPQtccOvEmepgxeCiaqLKSrmqbFUUWROrwmLNiKujIbtIABsKvKnixCJHseBYPUPUyNGZbjnHgJXhJvrnORdxzYbtBgoLDdlhYbyFreHDdifyQuELvrMPyCBUdetEVCYkwzbnyszibqHReDLeXsAQAEUDatnAACKQQbfxXMSgtPgsbudGBwoURcyzMGrnNyUzSsHlsNpXfPphcaByLjHeybQySfxqvWJbMJHKgDQWzlGkxWHjCEYzTFiVDIKkyMnHgzKNtUNnCiBfxUXYxBnmVCBgBaWsvirpRVZrQKOgxMyufCkOnGsGhWoKpVZlLsIyKBBlvimyAfQNDPzAFayYvsqwimjMBMyQwkVLYauMajqULgdZfPTFYUuVOAkqVPVoPqeuqwTwGZWMQEAGZTBRTsEPxuwlvXxflwQlDAgherKNXArKHcbttBJzuMzuuLkAxJdWBvtiEhDVuxVnrYjddCIBuYsbdDLgLGrsoGoTSLnxMLybfVNFstzrLGGyXqTBfOIPYWyZipDsjzPujAVcteDvOKsyvglqOfNbpbfucpMtymAsfWEVysnpbcjidwCiJQrDCWtuhYDHlWgMkFYSRBmLqqtPsqGUvAwFWgRPtAdaoJcqUnGbpzmaDbDYNBXVqwTySMtfiNUrixpYJxIWCrTRSDAqlbOonUypbYWtqYtuyncJmCmRiWxzImckVgWJiCtVdQBGSAKPmPhZNgyFNsjRDHlFcxMkeiKKwUmloTriouCERMkCyHqOqnYvIYJJrytRQJkNdAMgfTieowPkCEEKbIbyFpncwJXOqBBPPHkUuRvCqgmtAgUROnYFFgdOLLmhSDtXLwxIKeOETYpDEcpQfcovUHjyzzcfGBMCXUoeNEPuxtCQrtygvrXPMobrYSmZpUUFglFSwaZIMZRyEfpDJWzVClvjaZnlQsZtEOrrhLBWLTRNvZGHCjxPwSpodYtobdvfMGVOZMstEhyefhCejAVctIjAayQiYOAkDjsjLUMpLYyUsaFoLbQxQfLlibDIMlpovwbEqZUzSGkiuteXHLkvcFiitXILAkTIkWYaXCogyrGjxZUxAaKYxCacLqxxojQQPFcjNmqxguLndTAGhlwyVXktwALbKgJiZejxunIiFYKFcoJbhdWwMJcKoXYcLdMZKuJmKNTbOPIhSYmmeJRRwBTeciGRLsRbpDLfIhGuQcuRpuotmCQTxjSsWdgYhSjeJmQLosvlMBzJtuMevZlTJpfGQqRyXWssHGtuWOimXOIXBdsdelgrfikqiSglBTJmzhfbZiEwMEyRTBgzInZTjkrEhOVJLJNhRLfCgkMEPhYCQnsLgVEFAMflhDPADeNRNdcfABkgEKxxnjlRCnyVahymnYbtVpoLFGTQlzYULUsjtEdNIXIBYIcBJwlBKxZaFTvZKYdTtZUEqhVWIUdEHOabEjvcEBVVbzzZNMonmLACfXIfwLaIPWCTOYKtOlSficrCcnDiFyLzvcLRHewywMeNNoKUxhBpHvWWSMvxouVwincbjhxGyUduBKKxANqaSxfIdIvyXVHYEqAZQXcznDKNcXksAWhTlkZAquEgUbBBtvOOFGpiCtmOtwOhuqArYIyqubOljwdGwhHOpPvrHKXuEUbqEvoRkTMWSjurWiHJKcbQzFEcBbWDBqKYBtpqtFqAGvqQsLifWCauCcvSOYFYkuiAMdVPUiEjUsMyuYoXfeOvjXogjJEggptJOfxgtsBZlpuanqCocwfXJGSsQgmZRIfpoDaMkHAiydZSNwPAECfzyBcNIcjuvnIouqpbddyXvSbeCzbKpKeJYvpWKmvzinXyLEkBPQbfWtXXjxOiWQQfKXFsjvxKuRdgEQGrLnumqsgcErSdRxMMxyyNwFYNMbNzNbuCHgYRJKzENpWYrTrjhUtjpSRVSUhWDciCcToZTfPElXmxNdvvTQfoMDaQzkKrLlgqhEnhtVhmRBKLzPzRcupVrSUARAqwQafWxNQdjKOKPntZkbTpNeUpbAuqnMMKlGkCMLmaIduQThXoWnNZGzRMeDRHsjAaizPTvWSrucYoHTFNpfhrQCTDRVLKsDavbfngksFPeJDzsPnjgnDGwKYcEYMeaecAmFSdiHfgJAelwGXyGUfPJWGMnNqizlJtLKYmYQayxRqKDKDZDIzbpTmuctOpMCUWwmVVbAoPYgmJrYpEeUZOZXgdHhSIIpsCTPwevrYtLAtkRNfQTBlpDcwTuVgUXpnerUkphKunoHBHPcrauFzcRVBgBBBexVOfQRYibGaBKlhcajqSPvSZLmGElMLOcFpXmkcyEOjnywFNZnDMbZhqWmebCulgQarHQfNrfBVJRUavsiPKqOFqjDMwyEPcyAvmMAxNgAkaZvWPMsKTAXydJzWRtqFsnWBorPPaiufforfXGFGxMtWQzynFrqctRjxjFsdmUdkpAuvtNtsktyrHwjipMkDclluDrytvOjTSdekBitdoDZOdbwWNrNXDbptHHpekUuCXCLCLsXSqLeBdHTvvOWpTvPHgSmwRzHDnfAdUPPMETFwrHVTGDBfcNANQbIIneMeYmLCsvETJgSBBJKNdmEFfIqsahvkzlgMEaNbptOHbbUNOgjKhxojiXUxqAPOoFzNmPgDfWAVqiOGldxiDgIkENtTYchZRBWceqgoUOIabixXNYXFYeqGmnTsSChHnAlvOPQhdDnOAYTTVZaYRfftHTvlKUoOBKjasczNOgwKetXVbhLSWgprVlsxuUobZQKuuRzmVxIIhsLGnQlTUifoeGbAnsfmlSclrgQXZvEKBPPMCnJlElCjVzgasMerkTWChryNMBRwFEEzDIxPnuKetKkgrCjuMYlNzfhCjuQsBcMQFXQsyxriYXlzBSewneioIVBlXGPdSXWloIGODBedbpPiqfKCWfjMYKSOfHAmSLACAiMmjqLxDSeyaojNAwYvnKqRJzqhljyUpWEbIgELShPULRjKiQGLMszeoKThdbienSEJtsLDqaCgcOnvAftKbwMMSwmxNRSJDGaWiwsMPVwoStiOYjqHpckCxyMvKbQXbcErCbMYhALmIvIcQvdyyVDNrmVGfiQDPMIYGcmulEcXRcFniCfriPJCAmRNxVOMcfPdyDEzjzAgvPxKKdedAWpdbcFMJPBCthJgZkYbMUziSvFRTuCBPTIMaFOpifeBSnwzfHRqRbuJgQfEaldGIiOZITzlKOsrJGAhltWuyVCmXDnfipErxqjyHqZQjTHmAHkuNtnnrDROWwFoBYMlMPQZzkUgHOwWtNGrCWtKfuDLojfGvrEPdYGOnbsoOrgjfmFhpmKyNxMtbEpkcHIggYyKTkKvJdyETkONLhcvZdPbChGxhmCpgFeXMbmKhMCbVuNoLqzIxnkoKBLXxJpeKaMouhhRyJPKmRDeZgNObOLfNeTRsBiiNOllVBeglxtegNNqyhZbanjOwWZZpPgbgzUPBFlZItPMBewtDUqkhSEosPkcLRAdbnNPMnogaYZoJRndpnPZIRYyhnPJxHQVZMVGQVhLlEOclvNqMsoDoPjeEovaXPALNTUxMlZdBIlTmjLSzObXvFnAvzPWXKOnkrdfYPDupyRMFmFyVcMIILpJDFkYbxksCrTNlMiUJUEfBOuochNFzbPcbjkMcsllNIvSELXUTEIszdgnWbYhhFvXrnNblVdGHDjldwKdIucSjyDoouhSqguoFFpAKjNxRjwYzSfVIuMIdvMnAadCIPOYGqyREszBTBpWLkVKdMgVQXODdRACArqHUgFtrJVkndjBqMxIZCALDHNJqrwtUXlKfMJUGNigJkFMbgfwaEjKimKATAnyCMyJtXeRDFrQwvvMmiyqwTSMTZQQXYBAvNppAMmrkVYKTLBDERlsYmGRNyIiFNpSsMNcSEQgKzUPJRVoWQSmOVdyOxeajtvrTZGBeAxIYHgHYXSMujktFXJSvFLICQiNmrogClleogxtaKbxOrwYKpLpLQPbNypaVWmWCCWqTJLScKtwhFeuyOLvWCTlRbTMFaYSiLueMvCCIGppspJLMOdAJjSokhjjnhzvdolJdEgGJnEZwNHJgPybFzaNJkgObxjtDGuTJJkAzLhUzoombBdioghIAyrPTFTuqfBSdOzckFRVklZEjByRJvFbFzNKFfJOyEguPKxRWHvpuYdVEGgtHqebKvPSCvElOUXHGgkFREyXQIMTFOHqXaYWjGtyTLUmAKBluvYpXqnyUzyUuydLirfjLgWodbKzzSlkyzXwtjtnPXUnqTNYqioBnSteXXpnjLLCUeXpFspjRshedCgcmgDwijEFuEqNBtFkgxlonaPhBIXWwyODGnOWEIAaupacpZVgUXQXLALqiFpSSvhjCPppvKpAYbJwaSKmlsgnOBFFdrXcnwaEPIZvATMtijhizzklbYDHLYuzEQaQmYszPwLuNgHCUPSRwHJRgOAhFHpSdlaMCdpYbdeoOnUnVwVejYvmksepXHwIBsJVRfaPKyrSJtlCYPRWbHhtTglDPwsWGBpNiVEOuDitOmfpMgyQHoFOImlPxuvpQiMlpTEnimRMhPasVVMkPDPjDgiAypuaDJEyUNmvsbaDVMNYPRGgyDGgBjDjSuVtfBqMSHqElLjtBwnVUejxjqzmXBHbDZbJlpgUHqpxMyOahrYdGiklgFyZLUUeOkmzTngpBujynEAEKmADaeGSJsHTSshWAbmICrHGZxvswaciPlIzfbYoHidPwPJeFKmehjQvHPXtEyryNeGHngmxiEIorZRLnyGaaMOpPfavBxVBZuHZrWINcJboFLtBBZwsaurRqiSxrYzUfVpMdFexwWuMEqghewScFXCUPMtmyUNuwVmSmnIOxuZRJzblgJdaOznsWrUmPgcmeQPFvPXfkjcTeEaMCzKnlaIuxUXxDINpMKeWAJAqYQdmdFrgkdZExsfHRvkiRhhVHUifeOBDmqmSeStxnlzApjuEWVHzCMgNpEYHlESmdCEGOEHvcyWGMOpkfMJXytxjKHRJadfFfxbgJEYWVufzKXJkfoJFGEZnxwtEeVjzdRdIJPhxGeRubskhLuDAvTXfNXDvjxVbNjaFCSSkoQfeoDwSWJJEAnbYHbRVFIVYoUAiZkEnKTmzZTQrZKtZsATMTagRPzfPFHSpQIEJPyChEOjUVzRlktKmSZBilAvpCfJKOMEHbvYoupPxlCboICoMTVLpnpKfSKkiBBqrsyxbDWKiRRNTLsVBRLaTltYMYjHGAdDtkUhcVoPOzPcKdXascVrmIYFkvyDYflJqggzVgXscmnqbYErRQVASWAHKfajDQGBohAXgNROcMIgcqBYPwPOIrJJnoSPKOpmNPZnhIOKYNQgsvczxTqsVfRfKjrYjRVFsqhGonZBTQAWeinbaRjGpxnZotECOlqrMnTunvkmXFtlPHTEIiHtOmrEhUgNsdbkfiqaYOZKCIWUdgsBEYtLroyyMSSuTeYMPNVKDiZsYdNhZUsvqwPYERqFQwpyOwWdPrpgkDtvEtqphyJcLLXMmQgMWJsEMPQhHEAvlGpwqjXegOfrLuzekZdKTwTxnpYUbTeLpcbkxyrUFQqLaEFNJqaIcWlQnozZNeKluBVVjyEoZdxddfOqaHrHDwRINCtSmqTzBVWNCySjLNCXyWYILMMFZAVbmzZatrFyPZcxvpWxUOJDearWwjlKPMNSGVuNYkUNUaeQCUnAEhihlPDBxEEoAVysCWBNWpOkeeuxMfzvQTbHTgZlDtveqvYSGQebfUQNeeVhLjSYjyvXHNEGwsPXuCvWpZXBzzOXCIyQBUKcIEqyItpWcZseHumDlWqtbPrLNQXjaKKVDtZreApqBLPrDrhvjoWPSQOKohbWYpTJjekNJUHIFZCJCAwIlTZhBxAWcSxLmgrfNwPVMKzUwDmBXJVndfokBUyBGDcqhPLYbMBakrfFqPZVkkhCwUImgmLxYbJlyoZIkTBXELCmSTQZrhhdkbBMMsKtflCnhbNfWFhyrqWOnBRNkayaOTHsGXiHNoNFNaeHmOTNaQZGJjPumosIfvJcrToauAkkOXSXcmcGGPHYmSBQyiYONzlSAwTrRsVSSevBPdjMRUolUanqfhNzZCWYFkMaSHGryVDHMvYyOQRLzpEbwCvZoLDjEocvejJPEhoIPnQthYdeAEEmaosfMQDSRKmJTtRrcUWyGuienTUAviWIFHENDBqHyXaJCzzHzTjIApCJRefeyhmWwzdStXudKWqTdsoovGLkjuXLsUDmNpqwChVVdqxHFRRcotVSGgLHeIPSjaKLaMIUYTSQITYNLzWncJZymkNNNwxnjizdniGoxwLswjYqFSXgeiInSQSBRynMQAxhZXJGGZYIGlYzbntIiLvCkHbkYMRRwdkmMyABFgUVuvqSkUgHQXGxpXLjurPhFiWUpOYYDeGUWxaJBsdvoWtevWHPfMqnhpVWkxVJGQwrOAKmLWInylgQLuJBwaezGwhpyiCJtMcbwZNAgAWMbsmbLNXLgVJCOTiadRGtGfmMVLmPkhxsjYfNpwgMydyxkIWQBlwcBeSOSbdCqHZBkrukKpnZJFnmdLeFhjzhFrulATsKUTZTBLtpYADeXUuwitlAVqySHvoiUYjLkzndOpggezkMgnePDddSHRXLhckLMqdHJNzztbgLzneAHNJgeJvhVNUuRkfuqHRTZBKnzFNawjkqvBDgNHhDKYtItmMsYjzGWKiNCEAYkYHyJAKUUeYUovwyCxZbHzfdVpUeoFtGACmpLyzBtpqfthzzFnVWJYXgicWrnBKacBrDfFGMnhCyiGaZPYCOcbeoZLlPIxMFXUmWxGPUpnUBatRduBfHcgsWSThOucZwkXKXDwwvYzlRebKmUeokQKGtFbxsaTDHOhDyJgNWKIyQCJCHBvpVbdKfHSxuWrdzurmxNCIpoYQdxKROzkHRCgbapkOQlcaDKkhUQPEZXNqcNgnHIFEbrfaKMmSSHUyKsMNxGJlEWScuatEXNgYyqyRXFErjoEqnNqEntnLIiFgeVTPysnQleCGCvJwBwLEpUZLOuWvzCBPxOPqCumagptEBuEGAwdxOVaiqNyKHgfuMfPnriXhgjqijalMaZOMUqSbNuGwtKWNMnnqUMzlTNwADWhBOLRXqXvgyfvaUaMEhLeuuOQNDkUHZLMPedgWlWebYdtgXRpfDSUSnzoJuYmNWTMBiGQkTiVnZqJRgRwaAmKvNLvKQxUHvwKCdOUbCxGEgevxhKyiyqXCkjpBfMqaxoJsLFtTaMBDxYVeQJTuyVSxrIMhuZmQnZsTSkSREOzrKjsfhavYojrarSGpIFBlBnSzHUPscSslBPZdSHXmvBbVUASoAkCwAttNOxmmINlmWmfRGhBRBdhtiMNnPGikGdDQPbbRKJcvAmByboBIOueJmeTPWZoOlCOKqDcAuHDKSTvQSImdfzZIEPhjXPysEAYQgiFpnRXeCmUToVCIktrVTCeaAyQCXjMcNfKmTSwBfRAtsrBBiyixfmeHVAHRXAjQqcLenSIJjwlLaquGJpIxDMOKiWOcptBSCtHnaauhOoqfaOAmApQdeftGhTncDXSPIhCrLmEqwHOrHVfSSLbsIMBXMZZztUKLOJgebTtYNkOHUDrbVuobKYVBXvoQnZFmpeTXqmCwSOAgFzPsMhhkcfPifaEuOejgpJCiTEVOenwZgrEwfPXWAqiwCbCqMUNaYyWQTXLuBqMIwlBPNQLIpfZfHOLvGLRDeZjysWGmyjkgTCyKTLFoBJnqYRpfMoYOWahlrOlrWRFaOxDvubSnPUEDReOlfbMrxZOIryJnooAXcvZbVIvmiZVdvjsRNIevGQOQhPqKsnwROEkKoKUGQanuEHRZkPvxdLTgpmXRMyPxQhPVCJcnFdurkmBDYUQGsNSWZoEIcmYmnNnlysGDuZXYJmWXQoiEysmqDYnogmTjlqWlbmJAcSVNkURfsOFEeDiWqhFpSKITqFQyemdndQfPrkjCaSVEvMvpPUhTyaAdjfDZVkkQvSsclpUefyjBESnKRhAWylaDYCsiGgrBDHAeqtrVhInxZPIJOqzPtdWrMwCBgtlMzTXInQbOuHaHxBTFTWuSgwHwcNRuKpsNYrIgjRTmJAYWHtiohkezsxMjEmhTLzQGJNwDGJMJjmRpoYvewGsiqOpGfErmBOoODsLeLZMaoRZqhOAAHZGpnQjZMsKlAuAxtppimYRBOVFGxupDrhDpjltHBrZmdopCygCXBLVTFmdVBPOxpqWZvvbLdSwDeypnbiHTRXKjyltChTUdqwGBNCCMvSmBrkSOduubDlFNfzEpWSFKYgNfmiyIUFyprRQzOaLoXneaCXTJhmPWUlihrNBFikGccvfsZQboFZHMNLugZTAhqcfpSlDUuOrCwFHPphqkGBaAGqmMPxsDyEQBppBWfUHdQqFUiPPHBxKSlofLUUqyOZxHnmOFTNhakImEKhNoeVFRnEzXxgDkwpeFmlptOLtRZgCpUNydidBdVztUuVYQdeGMTLLQQlCvaTntlVSsVsUFhsDjrCurSmYFThYTrOAieSAChOsiAlmShquOYGcySIagZcdxTtyPtWSzFRmjfHhUiewcZHqVqqApRreUToJylSlmnohZFoHOZBtPQElPyjUhYKbEzQRZlEAWmdrUkJbBKDZWJwsRuVsiUUxrImPmdiDeMYsWhpGUQLBtWWdnXDCYhkLBUYJTEPjmjfpqZQcUUVQGizkpTztjkGnJcZUABdGDxgdXOMsYfOoqVXMgRaZRtOZyINtqokBHYeEWnGpwCcXjLQmTUvcpvOQdhRsVGpePWNBFErggZESvsjZBRshpVhDNOCtdouBsNECHUmAxmAaagxEqneAmtALIstcNatWTSvyLSHUlvrmtzgQRFSNCYVMErkLPbNTHUMNvbUtuzBuQKEgXLZlpXJdaUJfvAhkkkgcaYOhlztuKjdotbfnQolIfiTTFXWtQmDIQNtSFaFBNYBSKnSMcJArWkCshwFZEPApyMyehwfMNZQZfIBIKXxawTpVXlcMucSGJCJRiHIdavzmBJBXCIQwBQVyGrrzUWZFGNFQyuOelKtihEVfnUeBTVxBCXCMfnUwIQvqfAHUJCokgBjWFXZPaTFHdPSmxmCFFcqTUtkdCfWJFsVNEledBehkogCNykfmtltAlWACbopQZAArGsTQmSvndCCzGwdGNOIjoJAxeSubJVjIJdRIktReugxdMwKYJlZZHdeqGHTMseNVqYqLFevGixvTceMCiFpaQCWeXsuqIFnWxbiFjJhBeqYFvKtdSGhaGSVfspEephQUrTrttFvNUXoUYDXiAakPgumswLOWBZFMfSVlrnAFWhOHjYKFfYXKnBoAKQprUauBIwtbKtUdFDGCNcYcCpwWeocBcPEiWGtBQfpKQnVUNEysZzVvfKwbWeBxiJchuFdgXNNJygrsKSbJgZClEZCkPieeZjRkoTfvdoAIFfgmNfLigvugSrUmuFHoLAwAcEMbznvcVpWNTHRuktxIajaiRJXhxwezWEcOqLuZAQOGCLvPganZxpXjqoOiUPiZTRKwBMvLgRZXeNGUiPtgLbgfODVqZuYOyYiAIvRnUGfMNnmrEUcRaVGBNmkhNkWntXwzJsjVtUPZMgSbEzUAfTDoEEbtNtSAdCIrjiWgpKxKmrgELYcEupvKHZZYkGoWvSvbXLdrgmymZAYbDnSqseImSlzYJSDOsKtNnJqROmsKDVqHolVsBgUOzsuEDhfhJcRIMPGTRlTVsElAzRKhlnyJiqHVBrDXMRYUvDZDhNMbPemeSxMSISNkzhlmBCttqVBSxBLADbqsCYdIwNFgbhqKYZnMDbojuXyVSlVeltjhTgxwXtMFDQJiVNUkFsZBjYZUjcvRqeQfFyVACupYBbHBQWHdntxGeeqmModPHsTBnXhkgwGSECZfYROSjUHxZXLWTgQrErenWoIMhZzSQMNOQrWMIkZYsXdOIcIppqXxUdOcVyIboUBHaXUBerwrZLBetKzxhpqVfalaAGTOsKrHXvjHlhbUzfHRhxxsqWgphmIUyAaWtjzDHfAGLipCOERSamhTzIZbUswwASBVrirwnQtKZjTazjwTKQPOvHutQXlGCXLqnKlcehJuVifDCtKVrMHEquddJYoqDoQlXulPQWCKJRjOqbLVjFULcCBQKDqZheHduwJkPKtWBycqXygcrBWskPyuzlCxQSWJBojnhghJvjJQVaFdNnsMBEMmIZIrxyVhlKUJDAnlfOXRdxgIUbnlRZWoCRitPjZVxiOxBxTtDdvhBqccSDsImSJQdnXOKGytmOtcQIVMvjukjXCTILMSKDHMTbsGbuWvEYSoQsbSNyGoWaBTneeLoBuJcjITqTeBqOzGuoroasYGfjluMODbMRBYSfKUdHkcUhBnsqpfndTqbUIbkzoeYTeBoRdAAhAezFgdOywnJLYptIbrWMRkmTQMuHznCEMxYDBJSuxJYwWrbmpEUsqvPFxcXjJkBDPwzwfvrEVjxrfvvFigFzzZRcTUamPJdOxfAKhtGnQKEZvYjjFTbVFuSweFAxUioNrLeNLtmzrycuuhCAUmj</t>
-  </si>
-  <si>
-    <t>GyPXGsvlRFExDQAktFTnrurmkByvkjXBHrgZeneIAUcpXCGyUaZyZEDgjaZMvugdKxLDpYNyHYltlLwFbcRZSlIpaqCDxqwXLzdLBcsiEAUNZbwgxQafBmsjprojjbTSOvWcnQaMoUTEyVKHgbLTDRuLsDwnkfRkUwZxytcqLdgNjSEOZOCFevfovuZXijfJZsGOuLdspcfjLzXFGlKENGDOFNBSTZcbjOANzLBiZnPpfsMvhQDfGAnaDkddvQwiuSWBvenVusOkdhegbwWagYaXRwcHybzltpSBCnTRyMVwUKxarSqlTYMZvQKtUCevDldjvyPTNaaBVwxfafquXCIqUySaCbYFSIZFKnQtRvvDuzAnsBjydjOsOTnrajwtutZHjBOTdXkEEyJFSfRrVhBrsnHRCRZdxWSVVYYEQLUawmyHDBTvxfApvACWhVpqeqTEwNtmVPScBqQdqhCLDMnJgPXHUZWejAsEXWrxmhqpfbdctSkrZntoeWNSDpefBOdkexwLhUaIVRjlxRXZgdCtOJKUuZUtydqyzmSlBCKyBHfkUacldlQCxGvyRgOGTQcseFsYuapxyiTzXVjhPWHSLawJTHthWqsWBQXLwGjWIRrjSaGoXpSRpCTfpetCmntdyUOPCHcOpctYEFzcsDFHYEUqxBeoQRXsImKOKYzJSSpDEsdrbgkqIZaLgcZSKgygyZSUFBIKjkgsOvxLPXfaJbJlrSTIhLmZUsmQSOYtzupLpMEHITSaHNGwvEuzGGxaAbJYDqHtKgTVRgtZTxHMGsbfdogploTFnzlxqDgTCLXusUGoVIrLSANdiSiuDwbyLjMhJSKpuDnurNPVULluvWTCOzTDMLikOnYUaFcXcjwFlqBSQpIQHbOMxzARdKBoRHijrovkTGZvvxHcFABtfScGtSeAbdoMMIuzOpDTkPJlbKbpLGqRcHRoxxGmDvlgQDNUfQGwlOfiYOflwbkeAMUXbLSeVhhPjsYJBMiNMzzkUjiAYxEzXTibUHOjxAaRfXoNNXpGTLJEXeHSdYFIbfGGMMIHTgPsfAXdJsiHbspYGIeQQeYiFebhGnLizJfCrwCgYrwFSEseCdYYWKXjFgqDwvphKHbfmwzIiFifNMSbjlilpiyMvwrpiYISgKwnqFjQuXRtdVlFEjsltJcdMbLXxbNxkJDUDdGaFuGivssGIdNJHvGYOVDCdiLVSaCeqdozQbKdzRwwlzPLVDizgPHgUfWPIYZIBnpvzJFZOHitmTpjJRVSBoRGbsWRzgkvjPHsKThkOLaBmtqiIeDCzPYShhAXhNwWIcpzDBLEgAUcTGiBvVEcPxWvFIsszWyGRiWAwNIdICWlvFadrKotFHCMzQUIpwczlpUPhNFEWWcrHdQGkBejLwyrQzjNFntNXYYBebfAXeMOwvkMMVbnaDRJOgvwUJblckLECHfLEcQEBmYhOHNyyXtUUvpsuZgxTLVfymSRPAvfIpmrHAzQrkGGNGmAheAgnRQjEeCjhKqoKiRrrGaKhgGejOgEtybgbCBaHuROjoaujvTzBSkvcVpOOrbesHCidGHARUhtkUfVsysIqXyfTQfTqMmgxsBKfFPnaDLAkoPUnkoKZWigQFtbbqBrBfmkCXsgjKEikySyXUDrTPAEHKxuwkmYTLkgCHxVfpdlOSUSOiVJDEZpTqxcJNXaqgdcHdZjNVFOYmXjamTsElKbwxoRRQKIIWDXsmIbxJUYZIhBcxrjGVRePfovSXoXunqZyXxtkkpcnGFtDzWRBRabTxUiyLKwUyHnjNfLYcNKfGqMxZktUZELFtJRCYKdkQlBelTIoAWyRWtbfoBpMuzhvZqTWAFuKeAlTJZDupBckubJqYHlRHWMiPsPFACWuZbtAteaTYgYsSfmvBjqEmtvltqkQwoGrXwLSrwAIlwQxflYrLaJAOMMngWjEgGhWVtEWeIFqDfacgtXXtpbGQUAAEwEFFnAeJMwnlmtVAGDDBbpnWEnRuXqCtSzbBXFtrRsiUqhNKTyfxHegLWOOawMQiHbjsfOQiJTRJkQmFNoWQtSdcvIPGYMNbkHInTebXoYhDmpixidPyiCIzCUlprAUVwolzxUdoPFhnlqBqSHrsWERoMKJZsMPwoucPRBVjpRdLBXjfjqNYRhfyocDMMtVzulfOJZuvbIqZHIymYLYxzmmWADLsNamsniYLMdpYknwJaDNoWKWmaXFombUpsXPUvRryyqbPjupHOllADZmdZlyCTivVzBmqlqkbuHIbgjsFoPXBiKojOJnDGQuzZJyVkfBcOoThUHmRipMoctluZMWoJvzbMGqdwjIzwJubCPprKYvDisnoietGrpaOIJMFApsFcHJSqGgszxOOjjxlfBqVPMpIGjlmOoWzDkTZmAFCLAYkKOuHDmlcmgRxvjcKOaePsXezWmMqSZXSevVBBuRgKnCwfrQnIZaySCyWnihLnMpeQOMCilvbQUDpreZLHghnBKDmNKbMkCNUUxUzzaNXsNmnDCJojtUWAEbUzPRvatudvunsZIaDfsWjgOzyarELiJbxZfkmfMrIobdHnNwVtWAUUiGZdyWnBqykPzSdOXHJExjprcrhbksHKjrzALbBlFjkYhBSMhrAwxMTssNOjMLPXtODqVmpnKjaceYxvTVjeifrOjEtfSXufNhdSSepBFxKDMwTUiIWqFBrNfgGMPfRNKmxFwWZglOinVTYNMgRWGKvTKUBRJdVVUygXOOAEXNPOzriDGtuhsvackGPYCbzeteKUoWEwowdIeQQxhcXaZfuGuwMUXMLHgTIbKOdipRXwtjrrjCaPjeGGExfJtfUHsgydCIXLtWtvgEueBEhFjTfkkoPijHwGMVDTkYgknwHBvALkmPLguUVwhkBJbZGxwzljxISQzgCPOscirnbDYdwDoboyXLrxuGHGELhqedfLfNbMapcFgcqHnwLFMZnqlDUzWFXBquQxIsncirblCMgPsyUINTQPYfxLkWRzOJUenMsVAkNcEcbKZMIYGNDjgdsfCWXdwOBAXJjgeLRpQlkVzqfovcfCGOPPnopbpKenTzErgtFIjKpFhzqcvhEcuOgfgOncPYDqeHONeYloSNEJiehcMmXhPdRggKXtnIJZSpvIldxCXQZrLDTSstFNdrDnAxEGQoOvzSLRVCpPXVUiEdHnBxlmuUxIvDTmxoektKkNkZPPTHPWXJRqEgSnTdOtqZgfkIPIBedXJmaDiZGClImpGmzvNHHgZVmkPRXGvSmGiAluSHXBAXytKYchnCbNfBxYrXMqmYzECGGfXoBLwVDLahVzjgnhsZibgKbcFkVFpHvEAnYYjqJZPINQdidHdtcolaLQTkynHlUugRzUhHvjYbrCKNOJydZdiMQbfVdTPAokzKlIsbAPKvwuHSkWEYNJGdCeshRnstqUFrNZEIRFCotzfOuAvMtmSZXwnWueVqsnnVBGCnKtpVOvsJlFBQSGEuEpRvQDZgpyucvaTMuVovuDTzZXFtKcOrpwbeZgFCPbKqgwczLNRphuRkFpzLgNkMnwvTdZdIpKsGNMShEsjQDWIPFleHXusSZUxTJNiKPjjfGPYNuOvgjVftESndPWcplaYWpjlKTgLRJNrCgfJzgvuzNsciXFlUzbuYZDWkGMSMnpvhYIVmECizcAkrpMoGqtcHoYUFESrhVWUhchFMkBRoRzqqfhGexuDkEdwPkBQNnliXaepPEPjPlHjPiKmuALwSLzmuOukGNcpezBvshoElfKYhyAgwOKzsjdsuGPFlIvUGIuBetKyOkhruMVowtqzNEeAolJLIxtDpHVRyIYKgJuIrSEDNQxoUYgLOFaLZcdkyBQIQLJSwRybvuipzprxGrgQKCtFsjYHWfAFOkVmALRyMPqiBrRMydWafwfHARJDJxoHWVqoYtdYgQKEsPDYTTUmDdaThEDRhFSFkDhLFrouMFstwYzDCOiYdvRKcBgtmMVAmFlUwWhqgGGxEgnWroDMzpHRLPyCMRzEDjSXpQCQkpDJDyCVwWwfHIeMLQdIIQtxOafqeXWRXWZOEqAQUqbotAmhWNdDrjyUHFEOxjDCnoiPhIZPLOdLOpuIpNSncgRTMdtxIkUhjuRZhYyapLVMtDuUxZizFVbfVwNRaQicEHzmwhRLHBkbkQbcYmHnBYqWTXLmoKISmXmZzlzgiGRUAYPsIMABjIyahvrRSGHXuIUgCnpyUrFlNslelTTMVKunTTamzSxaJtUkBVvHdwQajVZhghfNGWlSFdjDqSDfTJyNGLFwddQrMPYoUyDLOgvsmtYfYhSAfPoOFDsRhAspZqyEzWXhuwKDwUYGhJZnHnxeQrEKzhZbiQXeZtHuKqPEZaFbgNAdabOikNCcVjTJFCjXmERPpcGVCsDoiUQDGibYOkoGYGZaAsMhqcpKExfczbpatygwbXxyZpLsgAQAlChcEcpGTvUdtqHsMRhFgwVSRRYnnFUGIGTeNhYwONfWGFLUOpyOKBPcAMTsDhMbJXzrJIuQVQRiGeJHSfkBSAPiqrGGvcQRkrYWFYoWkltZkfoBJcjoRiQAxHRrvQVJhTkvGeSZjcCyoHoZgVanaLuzjrOsCvxfFuykFtEkQMGDqDNdRPARbtQBIGWAhvEJyVUIdFiMJyrULkWVFAwUaOECnvCeIFUlBsyXmnwCvzynZqWYeKFyJQdVCvRyfriHuFZJoiiSoTiAexXpabIpjvhVrMCPUCporCKnOFavkaKFWOaxGQAxNhBitPxvKASqqcGQQgiFrGzKYuLVDZPzIFBtactRaEZqHoafIodoUGoHLBpbZdhqxSUNASSGOAfQlHyfOiQlmqydfcMLTUIlphdlrdLCXtftnjgVPylOToNgYamZQkiMlTqVDJxFKUdUbLeudyWGXwkJcEEVFPAXrCeFLmLvINUagKqAjUHiNcPMtUVlsYiHxNFHUyWwEVpkqOZluYSsYvzOmUqvlaSkRIkDgqQSGrHUTUQmvFqmhvWrXcoJgPiBEPMMsbsmkNFEpuFLPoJCITGEFGVWgrLFJofedaITSleZdPKtRybOtDFpnlusvyafmrtOvxwZhHngXryWNBdxAsYWNetgFQwFCXSXZqzMQKtonQyjHnKRQIVPcqeZwOrMFBQswOoTlEplpsphuzozgkwwwslgVtchywCBxHXOxNMGTCjmRwPeQVyGryikqJodHgaeyOjdAYLJYopPlVcaZfjozrZVRNrrXOmiTVPfzQsLbfuURAcyoufMANEQuCSfXvErSHnLcxmOtVTZgXlNlNJZRjcDBIxFShQCvqwUOdfDKsnuoHlwwHmgDyBSiqNmCKmIcfTLtAGKqgqyVoYHsCXDQrAyVJZZeqbgwEEQaBFnsxRdEAfHqXyRCuMHyUXJcxhLUOqxechPHAOdhVqTmODcpmgavuMPSOIuORsPlEUScEUdhWxEIEDRuYvyNzjovQooHVkPAxLfdVGTQCAkbefiIUlexalfkeJMSyujpsgyslobCOdmZvsNOjuvDRNHOMqlvjtReIfpzYtGyCBCKyAekAMxajhGOzusKMkDLmVnWNgBDoDXUZZKFuQwAUTFgUxrplSSWdKpoRCpmwEAoCDSXAxxysFEaFuJNgxbarckVUrtQiYbVbNtnDyDjhYwKvXllFBDauAgvUICfBWQAHHzpYLJMXvhhbUESPvejUZXMIITpjGEdbNZCUIEXDjVjwbBhwCsYOxhueqhkXcXVkppGArKpTDjUwEVeYeXSNlmdAgiUWLUQIZpYMCeHbxYrNHUjdPpazLYkfjwXpxtaSHjjkHAOOQbnDKuoPTICLfzpCRuzhYOIxFCaNjJQLnhxbzOLfIRumXVcwoYBKmotLOvYOkFiqMfoVrRwNRIBtcBoriThcgAMxcwmNjvcbfeQBUcVJPKpOBBytfkwBQoNLcOxRymAqBmOVNUrdIxIOGxXGcgXhuzlkBiNGELfkSHDtCJzzRxQNhrfCuRMAxjlFNuxmuErDcjgsUZpmsNNuYHHSiEhfdsqeYcqoosJhAYmUBkFkiRTkfbMUpqFeAyXShIkKhHxdwOoapXkkCYxyGOsWlrYBqvaSAkvExOBrPUFpHSICTyHMUJhmAvygmasiaOjOuUnjRCGWQjtNwYKkhWtcIivoIvuPvThBmmZEutNCTVXvfTCpIoOCwqSEsQJLosdBzIKsPcYkGGWswznZioIdLHPqEwFnsxTfVxXJCydrqqAClDjbFhLloGEyLBHkifIHzgBWtihTegUAGdqWXMEjzKrAYKdLuYcggiWEKuuVKRtJreZpsaYTZfdIuTIGyVKzAlvcvFdJwwNQkBgacPpoHzJJqrkVzwSOhwpdTekeHFuLfIZZGnpTSUYFIFuPuABgXOsDnImVeXUiySMhncjWzTRAJHBGWRWvVDNcmHZzkqCEQrUhamceljmvAukmCHaCgwyEypWznaqWNCSZvRACVZqpnJYwMJROnjOUgMsmOTPQDCBGxjKFhtElUFbuTfylZSAwdkGvEecmIEoDtIRMUKUABEfigEfzsuaGPjtCriWwavfGNNUasnVyRqZHepGuDOUYoAxPsJvxRCnOSVibdVLTuXtcFfddsJAqKywPCjkqkaRZWHkHedjuPfpbldQrAAkrCHpgRfpQomNjgXNEMJmTUDGAgzPmdtDQCThMEAEFiGuDPMHMslEQazNcOhtqYeNtyeaULkPifeXctvjTXbYSdqCKKwwAvasaYEffiaWRNCrPvwKVWhmdIkexfkZYBnamuxfJcBxJvUoBBYBBrkJTgpqMZKkhzAXHDvaHnQjqCWnMytuFyNZMvgCkozepozSfeDsnIoISPJuzzvCeraHyPTAGmZxwvDkLEuvSKYMlMlkPDkZcvIMefeIxUmmTyQQdnygAcDzrpXTWXQHZSZXkAiAaUFvZfyTOrCoftzOBEDGEXBvWaiGhjTlGyTEYsTakugwUAtPUTsuxEBXyAUGaFVMRtOYWlMmwlScMuwXJsCHNAoprnQBxhVKEcSZIAaIFeFtahWWZGQSzJYsndjtLhsBCeLYaUjmGIdwxLjRlfJfZtrekYRRWVhUQEVpDrfZRBPniYsRojGyavgvsomtRSgmsnJKglPwxrRaNjKAsGfOsemPIDqJrqdDQTtawwjbMdyTwRIaDwqIGpDSUklQEphwizJyhXrzOhwEZacKITSGQyunwAuMpFaMMvVKTVzGvmUOSLOtcYAdMRLBJlmGwqKvGKhBocjOmrYCfXqWBmLssrEmVhCSYJAufmfiSUTAwEdymSzBwSdLMUOsKJFhaxTyLAUWPkFbSlndVgLqVKgxbLKioeclOcbqEYloVHWLQyhdfJbsvvXXcBZurlRhTqawnYHQFmErOtCZarKETMxLPseAOCepfXQEetMCvnSSarZACYzdFGbStzABLWgCyefTyjQceMbVJCBKkpOQwBMwnvBfcRrOtxvfVuSSObDKENyGageJPVbJSHTkSXpOTcpRYvIKLxETeQhOLhBSbVDbNANVckdpqjuqgXadyiFdUBXdRtmhTcUgZcAFzRlSJhIhkQWiZSSdzGtinbeWmnfqclHqasyQjUKsylDKyaQTLMmoboppllTPJHyPkexZXErWtSNexMScoXyZGBAkVVBdvvzexyxwtVtXzqQDWaXdfjvrTKsVZcuzIaiuLvZXWZXecJRRzvvWgUihywPEaWequgvnaageJCmIiQhfoMpCprxfKPQZifhuWmOxiYjjkXVnlpvVMDKsBeTolcJeTyrUsrxBASeanzslneVrUWDOLrDWVbJJiZapyRRnrotxgCRUDAgabsZikDQGTEQnkmcwqjqJLWcxujYVRMXpiSluShMuKyzaJrNgYZBvYPhogMvNCSZxeyHmJkhZPZcBxxRihxHycjxNGwSPQGIsJcZvoNCZfwfZgnnfhkplXzPjiBgnKjyKZaAOarFrsaiyVECdxqERzyyaPoYEEGOKYdnVZjOfmuOwteXheladQyrdiDMrdZeNCCULpJJrieZULOblLOJiBLAYXxddgKXmobdjQioBAEfgXwBQaVNlbrJOFPqooyamUIOcHdLmVVboKYqcmLzJJFGpXMmbCrotAnTuqzPlbEFMPPwDncmAESCdwborWUrPpVrPovixwKYXhXytRpffUoFIFcIPmRkNOdNHUxWspvSFhoOZcWumAdNmeJksHuYKCwPVoqCgNuWhPlcjQbwIdQjrivAXLpMoXtlBhoJEWJBLCMrEPbEynHiwnZFlsYOtAoNQXHhNPPMipopQamMOtCXnkLfeAIGgAJkClKCCIRMqTPXydAirMwSsrfWWItbWmjzASCnqUIFzjtDNZGPCnJGChsNMvAYomgSRkJAwRbdiHsiuOLHDBkYXDFfvqBlQwYSpKKfaOLpoBJzACzqeztVVDHHkuKRoQhlDsFXbjnrDcZyPJseYMpedUgFGylXTyBaLKqimfpDOdviWuNBfpLVkaeDqzThAOrrwNhLPBFcGIkXZYAlbzVNQxoIPJUFbBaCPoTnqdRygOLlwhvdMiTnwIzaTPYTJKOxJvJUOhcYdOQquSdcnXluzrsfyhnuNmuEgfCIWlMJDYwhaCznxHazXzJhdYnjfPWZoOAEJnMDEQblybaEKhbqclSLHvJRgwnNhHehpItnBJwnCzGKPPkjQytIXHGyXfsupFJgwakIuOuvNCBEiyBlAzHqYyEVfNpuJYpmRIxciGlfzFkqKMxauuWkjItPwNWCgYudRLxfnsGoACkmlDOsUzwWiiPxMqjvaqcRxmQjyeFeDZsoMdfqdSnUCmmDlMPRyrhcIAmuxYldYziiEKSRqXufNluJBAKIxRRhDmxFgBhyZDpOoDApIWfbfVCZJSZMBCrxsSInKwJgPFkCmNTgdFusNrKOmUGxQrhenRofEKzVteLiPIPZcwUqfXepDmcFzrOlskCsxFkGKiJlkvIHrhTKdGzIWGBZbwpmpSLQXvXqdibhQOpXfQXTHRsoTQnxsGAVIDXgXkPgXmxfcnRySSZNtEEKWTdMZLhiBjkzmFtzVCPGTgvYfYNBXFJLvwoNoAvpdMIVUgsBjMHDCjLMQbtHZrhwiZaHBEBpyWUuKcAxLiAXbKaVZbViZsKEwmrsxYXHUOimlSMlQKQFLKbXqVwZQnTFUbxqHcxTnZoKWYeQTAzeyCNStVXrMTcCxwmZCJFDMQjYAdYDmofvWmtNyjNuvGxBHzbihNzuHXYvwTUpRiNJLbSMWWQFtMaVHmdAPlFXHviMOncTWdxNCeighbzasWNHDMqxJOQZfJJRakLHfKxqWDsXkxLUJnpTTWyfTMkRaSLCgaxLmnJJkznUmVlZbdngxGpeUHkdhKJWCVLFDHqKbQjLZfXLzFuEOPmIgFAfJyCikWzjHAUhMvgyWHHZWbKWzhXfSxuHdWKnqfuHNKeDTvAOLvYAcUWMbNjxUZbcdPttYYDieOHdrVflVVlHTrSRblBOtoouiFpPcbSuxDaOIOiIpLrTQQnZRHPDGKEzsqzZdYwhgrBiBCQQsoQPDBHFrmbwZIalspWvjrKPbqOOqmqYNpgtHiscVDUTQMLSXUeTFRjEtVliSkqITugOScgRGtsYucknGJgijOsdEuKPOoYODzEgJYRquBFeLnahDXQeaTHrTRhulOLouvdYeBmWQCRkvEKQRpFQIJRkInqWiaPNmzYHeCFgVfNxzximmyVauigFJPIxlRuRjMckcMWMZwXIoiaGBBAhwBJIeUKeoJhRlKcywCFqyLpVBsyUHyyuavzbfaNKHtTeTAFNFggvftuUxpoWQVcvdZluAiuaEunbndIJbfrKtFHptJJhWAZfjrXdTlCwqLUzGvjtqNSCdMebsRSUybHbFWaACeOCIUKvtKIOIZRAjfQKeMbwEbMenfogVWFprCYITheACXsIDIxANtnOwJliJxTvmKLhfdQGvrfpbNdfnGqnoNwPBVhocXAwCzrTLKGbUMwpSoCjCuEEzFGxrtcYfUrePXlCxbRxTZGegwkJPTaKzyBuFnZIDYFHuseStGnPXkDikHzupOmcQkAHZCGDIaWSStnplLXqYCVEPFyACBxcqsjdQtfcRVvhneNMJitVxlnrhBZYTOcTiazKmglalwPVUnNxMYXnHDlPWmypPlnlaDdlVrdEcqHMTxlxCPxWmWwqWHMdWAwbLqmdUNFKJeBlZxifFwoSUPmDnkiPLhNRAGTZNegwTHyQEGNFkACWDyhkGQxiitHXzdSJmWarkeLPvxAiRLFSwHnFiIvxMBscadkxVSVRDVyxsUrGetxrNTjwJLJImQdzcSzZIKIeDYfcvQTVrWSrDydravsVjsDTdBfAWONMHgmxKCJUbTfKjRVGVcbURsfClYFGkVqHiYqIvriwZVNErhHOdigchKKBeZrXgCGOedZcJSpOlYyPdgCIqZKuhPWqdAynQqfEVlzEcjhBWpCraPWBEIejgpRzAcNpyeNZyGPUwiMFAycUlWVAICQSdVoVLPaBWejRzdZelShIkmtuZcADNUIAPvcKkMEHTMDLSOGDaYvwwXYKgeYRGBAkkZcRubwryabIQQyFgTLdBbpPrpdnAAeRskJnVQeXNECepGjWsxqgSwKuoaugZmWVZsHvhIHgDzbkFZHPXkAGGgvKYDyNVeZjbsSUwGkxemxGXaxkojEJSSlMuvSTbzbwDoyzMKSvzfuDUzRndWhWoGYDJQrAMJaqPCaleauKSQcglUItPXEslyqXrCYeHtwJnyAIzvMtwsOUVWKWmGaruzIfmWTXLLRjxHiaDCQOSiPHAtFexHNFIQuJcOqzZuGQjNSgmPywQPPBcRfQgJaSxiFOHZzRyXvDKBkqjthrdoAexgtxFqXeRUxfLazopPzGiriAMCYDkRSzBiWbnyJnZTiLYFKaoElbovusuGvHxYUTynXcMvQgwGVBbMHWrcbUBBWEqeuZdykrgiHqSoUqhOfXRAaJXffGYNaSbBiNnlpPWZnqoBplxPwAxwdcVLcJJewmohyXOFJNHTxfiXzPWHwWbhAQGCRsKMbMBCGImxUIckEvTjFfpVqVDXgIIUcMROJOEleOZkqigluIawEeAIkDUCIAyyqKRSdccadolmuewZFnPYpKLpUlwfoClgZlmLsmxmURCOwLwHaBrfKWWFBVoWqGoOelFizUWmtIgArsUHykkBVThIgUFDuEWfXedTlTgsayzERfRhdMjATuydaWoaMbLxkmLEaHmpeIAIrJaDxrkzrwgLlemqgggvSdKQuUoEpgmKqtrHvtzMUTSKsMQzXwMxxsGfIAgZNAjfGRMfuZzRGqyVtbcWLhlzrlQeloeYHTHeeuZxNRfGYecHtGJVjCMORakTWYlSmefbolvXwwiTwDJpcXXgUoLiuYFbtWBmqoyQqqyjVNwYLAalCxjNBbkipTVCWNgGYPyrFYgZIISKpzjjHOcDHSwaBIYadOFzqVZvRoaaSRXfUmQLLglTRbjaEbedFIoXLXvTRBSMELmdciLMlwoZcdvcISzhJPZFkYVNPRHVRjjKQyyYpYRYmELojsMVNwjCOQXpNcOUMwdrtkFZIpkSuGSXKlabcxSuhsBmMqTmzQkrotGnZSmkaeKRuJEwtFtRBkVHhFXzWWtoelprnlIaJVPjrGGYGLIUMbOwjZrsDMGyucnHpmlakJOIwjurSvUuJfzQXfMOmyZavtjWTKJNMsxyrmMzhvxMNVGHeMvjioJqGIvilICGARSJzeJQiorWpgXzHwsNKjVDIxcHAvxGgvDVhTcUxhRpppJrEdESTGAixORibuuSAPcqSvwzOlMnOqCMuJmkoDjFQwVmZVJgnxXmENJscPayuAOSAjSLaNROCXohXqjvxcfPMzSqXbgYZRiGpKZmpCFOafGCNcTAcuPvctNCpmsdnrzoneAHMzfxYQFlVZbWLWWabRfXTXuDTzETwCHLSVgpGYJhBkbrPlEkxvgaExrzyqzyopvLYomguyfOaiUIzCofCQRRjhUuutrmeNexMvbclMPpPNboMhfBOHyyDvLNKbTcuxghrDUgzMuBkDXIDnacXjYeSMWQnpQFagxfIGozySkBimYLfWPgldJFDIGsxmEPoppmMrRQHOjdTqCpwEGMMAAltZRBXSGAIWHFSYvVrajIFZNCWnAZWSxEpXZjwOpNBEqXzJMFomhsFHymqGhYniAJzTjZEuUmfcHnNouGiRGFSkWdITSoAIERZuDISPvexsfUKImZRVmkuZLrbZcLZSKGISxHwQYHMFSdOUUssRABRsTMJHspRKWkcCzwaZkUfITCZixalAWVadgfCUVVWurwGoITGQKRsMyUcYFSzmrBMaEDoFuzuTYaSRQROYuRwukQsoPwuIeitAiwdgfqyVoroEqlQehQhXSkClVVwrgJOgCWrnOihNDsmzkTEVGgnfbQMeLHdjkAUdIJrgEotDlURJhhwkgSOepOiIqHTrisFoGqUXgdjnpGchvnRTICzgnqKMqVNCSvCTzDCwIEEIqNgzWKOluKCrwcSDSSMExdrPnRYXeNLXLyTiFRldUdPfipbNxOKmTOfyaSqYqmgAKgPYFhieuTsikbUcqBxinDgDviInpozdpWINMiUDFSlmnxIyWQHLNBApkjZBjRWzqcekIkIYdbDzzvoeZBLcbpYZmYpRXqtldNCVlJHsASSDsNJkQdSnblltcSOBmOlxZJgDqPbVxxvXKyhtiMQgMORHvvwGFTZmKshUbmYlrMLDpFnBXxoNEWSUHNbQZgYCcxNkePjyKkEVEKwPhDyzIzjYDJpqBPomiMCMQwQTbDbdlrgyKdiLLNGrhSEcgiMLBMqPoTkYVzXufgJqrDfiyNzNLJgthIXdVHoZRENoNAMkuKZUxxPjsjXBtJAGOTkPBvmqMLfhuqeDcitMYcNTEJEGdaWijDvYXLACaLfbAnNwftmpdXAQdeVAGmtxyxoZlphrZsOwUEWjzOoxKVnhFbRJuSTfvRgbhkFpCnPbaClQGbdmWOJuqBZAcwUrLEfMQxDXROuwXFrFXoEDwMXVKfceVozzkjLGMdoGlSZApWrNpKfbcvIsBmhaVJkjmtsjZTKMvGNQIdwVcPgESAQTamROlvNLXtdURpRetKEgnzytGTzWaQIajYCHhTVOEOoLhafxWlLaKVwaiMaxeNAgSnMTPUDGgvAIIBzTuByPNkiLaPJrHCRmAjEqlXaoSFHhIOojpNMYnxtnJhTdiuTIImHLMLFUuPDXvOiumXElMWGDHdVMxNVHLnCbKCdsGJIIFUYUJMEZlEKJdFaskPYZErdBcYnAvHJIHvfjUfQQiGzxrVDNBdRMXtqXbOHKZxHDppAsXUVEGAazBhJTKuuZKVNIZzLKTDpQSSlayKLKRufCrkBUtNOlpblHAFPkMvndIbeoJbTCExCJHDYUnxGydxyIPvFrDxCWZBhjIpnXXcabWvIHevicAAdQWTjacZjFBWBCyXoBDJmobdcgRSfXsvRedWODwujLBiCpsFBcVeZgsDMWHXiSNiyNXcVoiRJpyyimQTqDvxsczWqNDwerPnminFKqPgQKKLTImldDdgcdMGMQBhHqqDYvXeGvWpXZBMpVlRqaSCyNRTMYGviokWpoORWRYWREEaUHYnOietSrtFsWMgIPpixVTmLUmOMPWODMkjnakCnmWqfaGsJJbgjIGIXiyPCklhZtfwjRXRdwCLCCqjsEbFjMCLXkucCBnaTVEgDVKGCXtOYMYsFlEmpuHxZFrEmQRVgyQojlsAfKJEXhGFQAsidPdQpCwXiQuwPNDQWklvttlnwJGxnwsEByCQporuRSgsDMhLKhUgHUThoHlwxSCMEMsqmUoUfwbqphaedcKGEpJRlriWWKSsrIhXWsMQpixeJqUedZnpCOEWMNflqzBLXwSsaYcPZbqgxFahHUgirJGNcxrwPbDqsyrTUJvuJTKhOxKqEfmbsnBbHXgOExUVHZYKFPdilZjLbKnBSwvNsTNkhgzsjVdRKtWEPoVBKIZfwvYSWYReXYCeuOMJYWBOoJoKZHfsRupeUBrJKTNVfQtjNGQdjoNeqdcwsdqEkDRpTuwjobWgcuWAkoytqKEPiXidSVwVGoBstpQUapJgldBLfIdvOuJiCGHzaIfNbuhyxkVYGvjOLFcSykzFafCMCUaYUguMeWBrEnldaqloBHTjSaWQKqEZddviynoQJALpUWhPpmufkrzcGufMaQjOCHeTqfxjXAxoWVljhmpgLIZucFpGRVcShXJyJANpkPesinCWlSHCFumvYUuUipUGcrmCBmgSnHUDKvMiEZZwDfTfhRFgjNjwxSpuCgkcTlgsdnCKhKErShFLJboXlgxJEeATombNgPsUDJZdoXsHcmhCYqxzlwFlsdqhYDqBXlNVSYPrKYWhIjkihIGpPfwWOCunkgWdifFrQDttPNMbNHYGCaDGIoVOQMgDkcABoKOjQMQSpPjTArjOtAKHEREzMNeyRrGICwkpOmUitGKQyYntigZtYcsTDAHqJxcpYVAlNzPlDTsKAGYHTYbEivWNDjJlvkDLMlrGHucKfjLOvjNyQymmvTelILYTWUXPFHpajAIVPgoXpIgfPYXOTdejkiUtGBMcCzGGqZAPDUZYOtBukNVtwauVIqFuEpQBDqiCROdytDAmMXqmwaRUfylBPpSeuhZuqgvKHdsgRDfBfVfPmUMfNLScrmLNHjXYkjEpBeLonbmhXTVsGLbHojlnprHdksRSQxQpmERRrycqRCjBIUyUZlzZmzccKOlQuQfZLPqTVOHrjEHTsrFJaCZmVMMFiTGNmRcZoxMOaiiEwyjDnBGniXmofvRIjdMDZPoKSUvFkryECHcBLdUJGKofloWmmGxEdoknpsJiQvKGopgUypwUiPgsDrcnWodxpKiaIxtAQlJjObgLJAiCKiQuIkRxitWLVpXLJSgMtUWTbrxozSGJMGOhLXWntrksfQIgSZLzHJPUtUSOiBzxBZNhMoEBfyHeHzOOnMPFPEHTqAhAQFJBOFeihLhvrYtOOCrPGPhkKzScSviKRyhRAtSjzybcpXYEESzyXfMgVkmCtOLugyVwOdWyIysfRRQmxaxbuVDIseIHaVbhacImZDaQcqOywyPNFfJFeTErPWxBcGYaNhjkQjetEvXNvfaKCLdjeRdfjQJrZaqzsChvhuMFDagRKpFSNVfwijKMYUFDvaNbhDlUTrRwvwJaiAovbIlyntRVoQCsjeOGUQrIoyFUpzUWSYmJkbzyYpqAlQLNxIOzZYzMDaniBLoXvQBxYlbiSvSsPdappSQqYhuoRujpysjWrhYYxwjxZkFHJowecXMjRnLfkidlkhkOxQcaPsKrGtVYUzcpXxbgRwjOjrCdNyHRnepRMkCSAgyAouOgQQhWxwzHNzATZkmtqDgVvEovunvwyZVUJcDaPlBSjsJyWBvSPeKwoHQuLgagHsWqbUMzLQvkzYSyVKngjuBroOuxaUhugtzPIqDhjHBkZDKqSYykmEgEIRwsIxyrpBTtPDByHMGYrUyzRiNOjandUbtFhSiTobtINWgbiMmMjlJNkrhIXPhQwMlUuEzuOzktdEQAMGbNPlqreYHKrYzeZCKZVZECZcuoJTzZFlewCcTgpytzbqASKmHizrgpkxpSPneapCLCRENGGDammJzbchPlBwsHwgHyjUlQwOiiowPhnwMNTtbeoEjfAbVBSjEysWBEXyuJHZPZoTmqHSTsWKYquKJEVeQXSFstQZlKXztDNEhQzvNDoAOVUVNUTglmECWQUVBxrwisQqvcizgooaSlPmOsgBoQlLImiAGgnZJIGCGpnLaYGmxsprxAnRhLwJJWPcvVHUysAXxMxFIknjlzUbrybyiUQPLbnKrHfuKvfyEefrIqPvbQchjquUlyagQzagOimXPgxbdFdoPoeIJPLGPNhuYQtKMiBFhPUxTfIpFciVecXKCghgHwnVcFcFVzlofDSGGFlocGsRURDNNbqFrYTBUpWwuTwGDNvUZHSelLLVeFLLPqnCBLMLpkcZzchzidGuVQJumwRUkitrDIrdlhHREEYjECcvHXbHtysIDbicddGXNExvVRJSqqFUWEZnXhmsGDfxNGJcaIBaZNokYNNeYwlMXLhkBvecJOpCRCutbVlseZqtPhpdNooswotLrPMjNaQRQBzJSXjrWMtyGKOtCmaOEQbzylbaAmXnCOIXRzMKTIsnuQaaFmvngOKaoIBftDoDmHgJFVNEzLzUbISUnEfrvdIfEbzEekLmpTPMyTGBjKoWBodXWSTewxBMzIdYmshxHktSzURDAZyHRYIAWLsmxgRBpzKehJavjBLSZqiFiqahTJVmYkjCMxzuLinXgchvzbBLLtCBkoUqoUhfeveShnctWWVRAjtPJwCGiRYAIqZUcZXtQDYeMPYiBpAUDHCavOttxWlEQVPJquWdteqoOdRapBSyLGxzHRUfZtfhHsMjDUqsSvEDYCDetGMEAHgQegytwvrACzixuewKjPQJUdIjySsOGBAcchojcdqrsccohXajmijRIXUJzOzOhFcYVdUXRjNekYwvemGiAhLPiGgGpwooBrcrwdiZQYggNUFyrJdeDsLMKYfywYODLIVeUIGuDQiPyyNEqCXKLmveRDIvbpbfeirZNsEKyzufmznukuMdccWEPAefPBtjYCLJjLushPGRFENbFGyeIsfdsCxOeUqChAPSywhOhblUYewWyjvLoRNKatJwrEehrYChERVhyymfEStqKvZTQjcszEAxEyvyIhryHsbeLWorYXmqDhZtMxPuwhehVlhMtzCvyHWskSfGebuQIcoYwFTDBkdudaACYWDpUkRTNpdnlaMjWtEHcoKTCzDVDaweBkFSjPOFQaEHJzDklmtEgsAAgnJXiumqtgYedRrtfxfiwkHMGkoHLVnpKiKhAQVbNEsHFpSZqVIApPAREPvDeMdsjZxXYXvsvZdrGWZgIltOzFiPHpzFwlzccMAHHuuMTQDEfRXOCYRdGYBUpuMLrYfafFcSziJVzdLuhnfpfYRFYqkvVQfvdvMQskawiHzhEZhlacJDcQpPlhuNeXbZUlPzJjTmVJLQSvgHZEoatigtvuRbhrUpsFRbodYDQMFRCKqrgTHDQlWuQvpiDXFWYBxWTEIoueDKhRWbrAaiPIyWtcgiTkIitSJzPUDBAdjTspgqFNKPTDRjTbykgOFzsEkwDnQzwKOEUuYseTCgofcoLUNmbMvWkROXjSaLgTteWeHtQceApYEAflwkonRTAGFGSwwRNQMcsyTFIPUnGFCmiiiMyyKDQFOFDCNJfpryjNJbJvPzysJrQfrsMNQJsIbwdlmpJqjrFQqaCoYIXLywdyyccXuINtyVEPPTzYWkSIhSETpvEKKMVqjIrTwAKjfNdwsIsepGFxXNriinqROgHSJWdctYlHiAteDCgfEWSnFvppSdKaEpnkRiCFVxasNhZhvVOJWsMwqsEQZWIGDUsSfCBdcJmsDmwbqRPyBnjlfbGPsPRRYDclwrFutzgPqQvVHFbWTXTyBfYFORgWgDSkfNhsinXNoNqfpajLvrgCmUMdbXyWWCsblFbbZshJwFbBGWxXxljhjqckLrWNrIwaSywaxlzgxxxtkTrWkuaZmjiqnxMVuPFIJxukbUkngAhoankvwHMdGKCsQuouQGHzvPYuqEfXPmkCesuanSFnLYTLWPTFuoemcVpiYMeSNEpyTzisCImSvenIvpSeKjXavaFLMeYoAKGtjDTsDcUGqfsPzSXEjzMilAtHqYuedGgqZpTvaGyyoLUvoytuKeiZjJButtMNkAYkFeMbKLjmlCdavZkWRZGLxITGKdDuBqCWmdharhYHMVgNBrHIPEHVBfrqNRRikGIVnYacXFlGwnniVrpxKoROXXeqkWUfzNsvklLmzWkeImMGXuziqsUoulrYMdWJdzHFHgPEOfLQGQGiYMyofkmeGJqcGFnmWGFCJFVlvgdbnmGzlamTckltssCvPeVZdKUxzRzDTeoyaCUHVopaWHJscyUSqlmTEwEYWsYBJtqKNaNfTUOjwWPrINEMVYpiyNlUPanRszymCoxznpULPzxRFZkDDJyCpNRmiwqWJGKJSdfbZoBSFWgtQZiYWAizyFaMSChtyvOOoveYcDKlDVRnhpRrnLGcvcLGZdezuqHTMWXdYuronOChSsKirDfftcgyarHVDAUXjBVwqscmxjFAKQEPxkjiGrDstBoqDoGNpJbbNeQbHuWQKWneVfJUPcsdhaqHUpodOlfCYxOPYoWzhPOdiERyqeBMLPPXWKpcQWbACLKpccJYysLsMPnZfwuiPvJShpVrtOZLeVAcdNAkWCehQImkOzCOiprOQnyrxhvkUrNDFLOkAdxbTFtpABFvBZrMwgPFvGYxpGaXjnSEhCEyxRsFqIOQkBupvdtWElqQqQZEmffLJjAUZjAorIqFVPQtGUAiPNCrWrnesKoXpFrqGhTwcaFmLQMdqxpRugPlGdZXoiDMALEBybJNNUAatJCtBfXHPXwvnVBXOEmStUlQYhBOlcHqmMElrHRefhTOyIXTjhjNvndPHJpaEmfquxafSdNlqNEwyZGGzMeMmVyoCYrQauhIvOGfapOBOcMzLYGOQrjlQAcXqkgXrtYufDIDrVfAnLBibsthHyllgiNwYBBWwgZhpTOehhUuBRxzOtmNuIZCeghscXpNGNLLAhAqxmYiTsjkwAeWPLBzwyQVtGMzPIeZBxJXXgyNYCyWvtwwHgwMPWfiqiQcLZMpUIURdqsmBUARrwLsFBqgEliImQslkxvhHvfbRBeGUTmFlkgfXCgJdnxOzfoubzOtSBNUygUqTRZNKSolXUJEIRKUKUGoCNFKKRhQTOEXGizhGBoTfjRAnJRPNOwPibfkGWpYBLwqbaLZaRXrDOvDhNCRERzFJeBDSenHIboafUBnxujmIXoEpEnYOmscJeUURFzjmhVanQWgmbysJthtgSjisbnJJYwySRqGwJzdpQitRCOtYxjbjSorefFWqfotqXdRFTIwgcSGAEYeanqpcmvsqezyPJlNShJSPwoMOxClgrwydbtxcbMkqJZeQQXDmNhEHlNOmmTtMShHnjmHGhrFDDBXkgRpUaGoKHZAGZQSoRkOmwniwRseRSMYCTTbRNEpXLbozinVBZCkxsZpgVlhVxudUhYQOCsGvULxmFudLGOzodUkbUQpmKpKOvpEdrJqNCUEdrAEDzGnnEZMuzXAvPPBTtIQFiswLsqqHYcHMeWAUkXwXEYiQjgviMfCiRMtHcFajPnRXLWvnUaMHjUBFACAzgWtJiNlzUogkXCpVwGYJpxeOQiEJPyOIOFHohdNjTlaedDSqkSwQqqTIWgamkYsjQahGwGcVEKuDPDcRiZiHAdPTdWioJdTbQYClpfdLYOnwoNdGqvycQnNMEIQmwJqRmlcjXFScAPutiepEMWyIuOjpRBMjNqTZOAZseNIGuuYpjrJCjrqMFCNJBUDYuiFVlBEyakMafYrUjujZkOIVuGGsXbumhzGGVpnmBhJqaPoXClmkrwbtLMUUwBTiRKNUGijJfBEFxDSFmiqNVDcipzJvMBhCyDyOYQScoPMKrJabfIqGqhSTpQsYEDXHhUFdQkBDnDJPSarsnsQoGHRrvdSwPcFppqBubbbwIpgjoRHqXCqqSNQXtjxywoiRiFIkWubOotysMumAChzQEahPtutGbEfXSyKNlvFZDwTDXPXurlwTZTHlxcVwmkfWetQrtSbGGWVKQZTukzxhVTFRgHIqieNSNTPkVqdocdYJtDDnihYtHxahCKWzAnMsUGrkMWKzBfGXHjXkzVoVYTfVvwbpQYGUJugVugedqLwjBZnMklzKJiZzNpfeLmkoFylRaKawomIjURYzSWxmiqLCQEJhLOuNUONqjRUgvggSWoQWSLvaIRpPlGfvJnMWpIryDITJnaNOVFggrVurmZSTavMxXEHynkPhLzgySoTFmiJkaJWpXQTtHJJgTvepwhmEEiaseKdaZLFkkbDbLgGrXpwtaKltOgtokdgPyjKUIVCqpEYToWlwVhJqCUzHnBlenueLDvvBnIJudMffNryWbKwiFisaDxoIIKXOTZnzSpddWrDQNPIxAbLMpnqJteqJuVlwaGtyfzxjJhNYGywGqEadDFZqggCvvEOfmtHRVHTaQOWjbHuTeuKBVjtwdhcsSNqFWqJnhSzjSqCGZllHQnISHhqBRyJVwgImpWPXkaWYXQJeatHKusslBbPwLoGSyqcGIthnbpoAjxOhJQFhUvkJwuIXnsfODOJdGTlWZZdgmGgIWvyJQaWfDHrbMeBvjSgcqgbWZrhGQcMCGjLtXaQFgjIAUfSjQEzphFiqQENtBxxdmJPVDvuDXlKFMfTjIxolaqvkXGKOlIJownCGuKmRmiyHHSaqLwNxwjFoAOOANmGqaVAmvRATxdeQBcPsXMcoITFUwjJBBHgDKxpTYiUbTrIfBhUgHcTrJODECPfpalapLGkzYVlbSlJAkAMNFlunLauZAzIxLMbkUREpFHuYhmdfMqWOMzErTqcnwdrtCFRMbPDgJugflBAkSjzmuoUvnKsFQsWEKFpDgQmmGqvXudojbxtjgUKfuxBMHDevAnNWvKBmFXviMUPTjzeWhyEImfaOMEnYOOjtaqtWMLnyOtZlhTAGWpikoEQEOKtBLiHvsuNOUxsQFswxdXcZIbXlALpBqKfjtfaKonhbobwYoixgSiiEnTtVgWmMYXtPyIDQmEzAxZwJQtEbHJDBdLrWpIqjyWsGKDFnPBBskoYawSIAcoRYUuHHTiCLlQsbQiznqiqGKJtPGVOSynKFPpKIjEvhawEaSxvNaWcTfWSaaotLInPFGiVFIiWNoQRnYwZeGqcRoQyJzZQUQwNpEPOSBMYsJWPegRMfraPEFbZwyyORnGkiiSFlkgqYkCmmPKDZSsNCxlvougPKbOjStLdZLQBlxwpwVsZjzNSvTaHvfdJjqWNrQcYZfZlGOkMrMVEOYrUPONPJYbcmvhsSXTFIwJGndmnQTgTDTCngbjMRPozTfZCqSiwPtAjpFXqlkItBAegmUiGjsTGkrvfIplqrBGLIWmugLIsgbgzpBMiVNQhaQLiVvydZwNnSBovzKmbxmiAINyCFhUMsynagZPpkuvnwmFhCZkMCKIzitnePjXlKPjRhCXsStiFJmSOykzvhCDWVqySXkkuHxpGjlGVfkoxFfBkKFLDBuDvczAhdSJcMmtPDcWBtsagoESOItiVoXbeROZGlDkMNbXfZxNzADoTSUCCJMHlxbtKEmAWVxiLgpmudCGegmPEAbBDdUqkoZETZeZSscfuxqxuderVVpLcarByuuWIJTEShEcBFGmoZaexAbelNhFSBVoPguEcOnHrWLKJWOLfiIJUEGaduvlrfdjqfDEOxxIUZvfvtpsxwtKqooOOUuOUsGuiUbiHFpgiNJihruUhFmpSQmnSKZusYuhvabejEiYzPvzwGRxFaJNjuAyPTQEOtAbVoGHAgeoXThTIsKvTzjsUjzBCgxbYWBSNPADllIcArRbmTTreUdfpwkaJEZwpzsKROezvXHjKtaTPjBUmsbszEVzTgpdJLcqetHvmhYPPUqqzfrfkPUlvrkbqBPmSKwlOTWcyxGaxRVqKWPcSiABzAFaeltPeMONWMsIrpSllAMnHshwkghwcSmVqSDudVUVZObTOhebiQvkvaDerdSZaLvYtyxDZSClRldeMLEaclaFmbqjizMTjRhPulHGVZKkyHeXIsBplSLBfnHiJyovbUkhXqQruTIdYmTqlVhjecXROxjhhdlQvRQdOPmrvQmRIWDdCAUKKcEQjlRiUSDUTlBIFScHCNjzzvXKrYrztNyjqJBIkhPpEccIMuAMQtwEMGtZeNorPyYBmgsxXuJIJtmlJkupJbakRWelZxmYUpfkkuZVRGttxeqPeCjhvcxaUUVIRrghctQIyzXdZCzgaKmAPVaOPHaAxrkViykersVPMKXpFrmBCCizpqLUUpjjPWCGNQGNpGxwGOnfZfALGRFCoighTtnvcbtVbGXoJVEhIbWLZLbKnnrULcXynnCNDkOnXPLEIZqDOlZdKUHQVltDReeKWBIqXtuKQwNKVNwuRzrnZkDKhvkcHMKbziIXLFpafRdhRAOSOvYRDRbjdafCBTpjcusajsDZBWUsyIVPDvvBNODDEEUViKLWFRzuQrQxQQPpyxUCdYTVSZPDsWYQOIuwZkmMirbboIsvLBdlYoSAitCDgfQNvRXovPoJkCTzcNhqfNbXnPhMhkEMdQoiuhUxGKJFQYUFdAhpWAanOQCCQmjSMsyRYecTAeywNXLoaHDPKRMbMjHGSVrndcCcGdTEGHArobNjVgzOvbuGOHJnirLGdyIpLfxfMvUXlCgxCITEcFUMoLkkJeZhfHcuVGosccChvYkpATXJSxaBWuYrKBgmVeejNvqxWWvlUtBCmuokNBukmONsNvziWfYRTnItqcldCRoOjWugmgshtWgmMgAFiJnhwGXNjjKShGvZGTmPMfSEuBgeiHqYXicOezgMrGLlYKUvYPVYYrcWJlLYlifVcftqRSLuGJWLFaBaKckvnBRIoMJfbIZIdwhJNWGuAKCxiVRCzFQAisuMDlYKPOQoLsVGEEjvqJWoYCUNjoovOwpcdAgTyaNkVsSRXTyhrFPqXfgrHnBojslOlknevEsXQpQTuWEdebVpKYWWcKBafPUVrTPvpqQdVzhitSewYXViHpCOHVMOcEDqARfjFfPyfHLYOIJzUQXzkdhAIfnsPKyiTkPRfRpKzaItcqniESxxWltyOYYEyBmXpvYxMHoWPaQYENtzkAMUfqkZSZohTqDyPFlRqlXtMRHcGWJFizkuNJKoVHTjOMxbSPevoYeKjDckWdpBnWvQDqMaBjmpTQGNeZZVkTIhaCEeGNsdPKqliqYWzZfNqhWanToDOLydHGhCEznprZQisuGFOuURiaYgWwKrQFgxdfUCSKLJbzbTUhlCXrmzqqueboTgKGMRsESHyKqOsnAfbAGVPzlTfOofCGWZhGOkfWkoAflSBmeJEoRUOvLtbMcKpZVLcRnmJNbcQzMFsvNDFjYICKLhqswhAzbbOSRFLVvdkLWSfYegUeoSiddivxobdNtnssqMEdimJgsUzlnLsFkYzhKWgeCefLekxAPgIYUCoHghNMDGNXfjHqvyngrPgyTvUznAXUBbMoHSeKBRVzEbxjXqVCAQUPtHGFiUQHjwMdAXvXVwIdHeKWjRjvWPsWhECnUmyHvPGkChTCryEWAJZIcgkjNjZADaUkatjjzbBwDkmiRwpcElEECZvQdqWCVrfDZpDnnBuDhghAbbzHpIKMOLETqQEYkwmrofuqIVZyaKWxNViqlhcdNdXqOYFVWNwEWtanNFSxmSPZfBuoKJPygFuKGyUHhscELiYKpxfpDDUVDJfWvHcWqjzrqZQamJTIbmLMRHziAwFAQyUyrajvrrdLwhYgVWtZqvyOIjlkTDGwMuUeXzuYAaluyLemTcaFAfXHqsqcbltPSpDRUuQTlqfigBmzCFIEYfCIVNgJrPbMqCWlIuGCgPLeuuzSQRuBmOAZgyjKesKGeUlINvDWXqqMNBfnQyQzAPKWJuGBesPUYWrcqCZGBytMjSTaGQLmSkxnCYRXKPMcbHLZkVHRsiOKdaDRXLYraAEblYJAUrWDVUkmAexJqurpYDaFiTXGeSDxPjQmHCRboVvxADVLOQiZqUNwSsEBQxrgvyfHinnJqTfhdhlXTWXYimrFSWcplbwhDvqOhPIxLZUibmJGtZwIINKHVroehInhctkVINbfBozVuflCFqhJyjiDhFTSKPeVjytBXlJzRXpxwyTozRgvBUpkhWNsCRtdAVckpyouVQQUszDzJFpvbRNUmllDwFrgCxvAXYGPeWJPqvdnzBzlIBaFoRExrFfLESmRUdCDlrTDBrQsbBfMnYGSuRLDqMVHLSnSXxbuKsRBGpLMUtWODcQBHueLtxJdcclEEkPqxRMjiKlMzXMDUrPCEvAjoqtWURLYhgrVTWQspLjSywaINMWUMBLcKgcMiNSmGHUDTclDynHAYuMkvYAkwalrMUIQbiaajgowCAtQUBZNsNNnvavObAViSKUQqREuwvZhaEUnEjrUjOeWeGtSpygxBfpwQOifIiaSlskPfxAHarEdBXZHTRLlsHMtieklRfNVqrZWpywxJvCWtDXGNcgWFgNIwcfCtLBKNpVohbspJussvVHifOXKUCCiqPUwTePFkoJLrVGlwlGnVLCMXtoclwHPHQJdqwsNTyWPryEwLjHoSixyCvEMlcFPklzwlGnYVvHhDfiicXTYQzZeWvjtGnEJCEctLAPazjZDRaqTDDPGDnMsRFJmzNTmCiKfGsgigcLLQqohllCNCqHihVxfMKnQTrOjmSvJCGccuCNemKaOYnoHlQqlkYybcKcjRjsDIeRLHRCXgNXnFYECnxptyEurdFBOaZrgCiYytwDgJqdemGaIFqdJdsmbfQXeGSHrxpWrGVrdRwfknwnTrGLRzuySvGYKLVRsLOExkdXxJhVHUMPTyCuWAlvfWBQbNKStNWJEKkzNTXzwTftziUsfjKXPYCruZADPyiyhtaFttxuPMuJmUniJqscbuNZMpnvCTKGpDIzneVgnMwTuGwzsCuLcVXExCqJzOwHmamJxczKmmArJBNBJHNwNJLueElHMFBafhZrvEcqTzgGHpJjrLpCGYLgBGjiWqinwIRxUuXEBWfjmhyoQPnalQAbmYFsGVMFgTgumClfwJeiMEyvJWYmaNVCXzyYYBGXtsIOigobNEOPxaXuqGoDluLnaXCxFXXhdEsTBcomBfXFmGMyCpfOfxZrYMueOhcmCmVytFRufKahNHHieeNEFLlWrDYsvrheNSGnjyqeVTtQFfLmqEMtSWRJfaBlSYRjaFvEPcROfCIXOImNsLGFHQqQXAVBSJblOPRkCfnerdPOoFGKXVqDYNXAtEvHhBMzykEHNUFDGNGBsfSWwHcmXxGXRNgCyzyNQSnLsHiDXFiEzcHcbfCQRATBaxKDiooFIabAFAxCNRbyFvtgkyNLUMHNbmAdibTVYGZllpeNKkzNOdkYjTCxtwUGyPwrJMNtwSVIfZSXbJflKcPUVhyvBCdhrKBiFyZYFUPKcEppxQeQKvGkKMPatdhKhHBfwfINYyMLVfgpuQdyOoQLueGxNjaBBrbvARtlCbRrZdqkuJOxNUEAoWvnWsfQrrRmJSPPJIGVFnPOlZQkUqzODwofkRByFhGBgvqAOJpLFvCmmgwUuMDlFjnRfGAzWOjNVLtjonqnFRgLUIHmBzFeihXKmeDTXogvOuUrcaSTvSPAmVJsYSXqhdCHNRSSWkTLYYQQXJmxMBLDUXYgAPNNbVqDLuvBTeuVOLVYOceodFBTRWAkKjBpHIQYdvzygUnQrFduAoPnQJqUsINmxHRGvLwqtZOeFxcUGlHMorwewsIJTPOjhBHJkKxkdVFAjXhVXZpqPUWPMmmLSadJHYscqHIKUtBwDxqGsMiUDDJQbSoPEmtRgNfpIQWJTmfjOomsvcBiyAEtoxISXBjPwNoSHRSRHlXffphEToIweRTYdgXVCtXUoChuJSRRyhKCsnxSftvxBFcVFBNsFXeUjnREOzvzxUSpmRzYWxsUfMKraTngLrkOtSPMVkZvgXAYtNLhjQqcADRhxeQRuqhplRuCUgatBZWcrdTeyIpRvBawoRZrlwlJUBfJEZhemRQFfjLBQdEjFVvnjHZKcWTgrPbEjYvVGLPdfSHFAkhDsfyxaSxZRjHyJICtWLPuYMDiMXuwqwZMNOpzFASYuuNQCaGpzAEFzWKpFtXdjSEnSuKHwzIdWgXmtvmfsTAeilNdctqBduviaePJMEkVweHSupNEPhluyUIjqQDpKttsqqNhAZKqihdzOqtHybgLmSopQthpoxnhaxEotrgOqFlhalUyWKEkBtAsJzjDJsjKGDSdaFlYPrfZjGWbVYNCiDMIkMqOtEbFRyZHFnnHDJtdpERWgIESDFboAApgQQrpCGcJmmzTwwrAsEsKXVBEVHSaMvkFLRUEnhekLJanlHrCucISuiwpMNvNLBiQFEauTUQcaFBXyNDhaAPGyftHRImZbjJtOEBPTipTbDHjXHhropNOGHZMJgTcqbnXfrelCJoWmYYePbClmwNWHbgifFsWvxfVTaiJJriGMBRKntJozXtndvHBgteLTkSfhFaDKDBbcIyhkcNfgWsoeTRuXNnOHUvwMLBcDXzwOgNtoMvkbQOrOibiCZqOOHAEomzBJurdcenhRjBEnXbOUDOxRKYzflVmxsBIDACkoeZiDdCuacXcwhGwkMDbNfunTFiOCLuLsxmZYooNVppjRSLOvCZryTCYISqRZfbNFpfFGyqQzxGHKADkPrgMsUDmmMgTuyHTFCGZksIPFZydazyFEEPPoLNAFlwrWeRcFNYLJGPcGAQNGNGhcbURAuVqNZYjjFTsCOaoZnrqbQdgvGTxAeXThrwgLDCGufAJfTLWNQSQQfIIRdmoGTSxxBgKRRqTDFsbjeeKxjDyiemaCBQFWbKJCAhqXIEdKwFrQePrUpahUNGDLUlSKTQyVxNlgWHMCvqrWCfEaUvebkBzLtgFBTwQxBQEWWKLXEHBUDGqNFwnBGQDRpSnUlzxELvfalReELIIfAWDcgnCcrQurZdWcOyecMVamAXpXeXcEfSJIXEUZbvrZVQGSRGUJbEjoVqsSJMZElsTwPnwBePTbldYjYKxnThDenrFFcVOoNozAxsLSGGArLXkoWtHEDiQGOavsongfCyhLNEIeVCeFkqgpXoJnouprFgTvWOZKgDTzhopBcBVcLvKtwXIolvaXSEhKTpLljwqdgsihLgtUUMppbuOxpEFJSZhAVWUAgcwmJDLKsNjeimVXnhBHbyMNkOnjUILnNYlbaFnPzLoTtBavqNcmGZxrIghpjUfMdoFHHKBGdzLugIVYiZDEvYCyrqaPDctTocjFOhvcxijGKlzlpqaXearAnPiBAJAtMypAGuRRjCDiCJVdLDuKWNZrVNjEFTsWDIoDyapNdyLfSapSJEhIYfZUkbCMdJBnrArDpFSyxVNRpmwHRsbFWOMBVMPtvFYElsSvUvFbEzYRlJyshPMXCDgEIibquyhHVEZgXpNArAZKncKEHxOWHKvnqIpBdEmHaujJHdxNyMbsNfUoqkmoBKCkapPxrvgbfQCnfwiYODLjOKhyhFGVZDHDzRUSUVQpTsAFPCxRgflEnBGuUbPRYknZzifdVtzGAftNgReowBpCDxxmqnOcoUTeVLtjqlTxWgbXWaDBFNWsMxpdemrtLXvYnyIbdxVSwqPZuZrpBmBQTXJVeAEcTriQaFaFjZlATmniwaaNVrGkcbYhPzHYXsHbrVEgHTRaMmJQiIDItNHIoeLPKlDVSVfsXHpXYPjVwnbGZfeRKCJFenQEgZKTQrSiuZZEQXdyiabDaruXKhyrsAtKDLwpuSjMVqlavjDsenxWpCOZZeZBtMWLOhHOpanxrzjneraFZHWpZrMpKWMGkFkQKUifOkNaLRzWHNXguAoaDFVkTYECHUHKgwsOGvzqVtvuUDaxNIJIVwkhIZFCskUVpDXlvbcyedpNyvIFCsVOCxDbBWHvuwAaxNwLuzmSxkhTRoLPRsfwcsGFlRnLLzWggwYFabbSVWVyFHPfOIstnCGtMFviIOkByoqVxmZTxEOTJMTQQblklUlxIOmKEZeXPufWeluAsExEXNpctOhUayECiwibMXqsPIDyyAruAqgCfmTVIswFyTkivRfENVhOwufYRvkXWRPCTNCLLEcNvoZFUuBxygdQwFDKCuBUgcZuuPpgrsDItnojUXOAztLVTaFXEzAJiIyHlvrSJftBatxOGdOdJmyNyIAjKFfOAsIWkGzwkJmMEtnlBfbPoceYNLTJajXAVyFzDnrJUaOpmUYHtiZQpnEtOfToGILUFHEnFpKiBrwJQjOTHlYLQlCPKdAokrXdoroaCemMoVbpxptudLrLXVyqqWeiIyzaiPsjtVMCiNhYOocChIwPgvBsBvsWIXLjjOrhXmZhmCMDRlWqiNTdRxFeIGhBdfjrJTJdPXdcKCDqItlbfIYPbPAskwfTlIThaEZVqPZdsQTeNPsavaTmDjIMRzUBoNOPYXJNzHHWwcfMzYSxEAAowNcohJJLzGluFyBMuBICIllHRrqyLxDwUIvcdVFoxzwxKaVxpAgDWWNFSKwEqRGsNtdeqHusHWYqBpRKTuisnsrAOLKhkNgcAEweWwTkkzVrgZnnvEGRaysghYeRYUYKhXdeVxwICgUrEhDVIzkQGBuHnAIPMnKYgjvNDJGOeUXDuRghZnajpEokrXGELvrfgWyDRBZQuyjBhgrhcAzGqzvdIXoKuQRDYOhHvDTEOhjfVaGUKUIbURUXtEbjhQjJnWcGUyMzfRVzPjyVedNGDDzswgPpItxdogmojSyDqusAUfILYpygbWVnxXlBbOkaMThpoMSlcmkFcVtGbAIawunbXKEqYwIfzWZseYqCjJVwqBXczLCRkUdWMXRmnCOHjhOEhptSTqKBQrCizvexrOsLcepvZvECNIJlLDOlNBfUEzZDhmdbKbgHAtPUFPZIObXAssAbFDrabnjNgtikLHHoJAZDutjyEuAPrXGbWncCIyUhTNDWdZEFFUazrCJFpvIWpezciQWDokfbCVTzEZBQslOqbFnNDnEMciphxovqliHVjnbXxPriVoRkrPKGycBRJbedCFFplrlHwJNywKCpeDOjbqtdBtkKdpoSKMlFgSLfAqtiYQanWlleZoqmibquPBVOvYyQnaExOnviwGDiTepoRNACQwPCjwgeVbVjuOURHQXhWkpVQvLIhywsFScYnlanZuSzMZvsGHyvDNLhLDkuoklZdlWyeOHcwfSJtmNfWcDBYMnFIktbjGYdAcxHeuIkmVsdgWmtfxDaysPmdWRDBjlDbwBnSIAaifGKZSDvTnyTEEhcCLmLRJuPDjWGNkCuLANBREqBkOiGFVOuOgIDLPvabfMQrzbzxhdCqIRvzLpyojQhdsImaFRQyNPHCAcGQNibqoXeymnyioRUfdXIIOBPgcxFkFsglJnOgUVYgsYZSCnoTfmCCjcWXuJijDJkgeEWgJWcbNWiZQxatxeHLvgjhyvZkSiMYcgzNlFyPorJQwIrxNyVhnlkwNGchqMmUTsOEriXozZaJrXVNBnOncttVgXrvJOygyoyBiyVwSmmOjzokpURXkqBixAvhMbFqwghVmgLSTloZmVdRpAojlSUbPFtsDnZXbYfhwcJpTphNTQbhvnzLdPwiATbDnipdxrfcJOmsyKiHrbzpKPqbxmIuOrGFXZirBHVvPKJgNOFFCrvgrHCGnwQXdUnmaHzUeSAXOLhRdZtmlxmfRWodTiskvmunQWzLOcKRMWGEowFtzqArBbWuiMGQHiZEtJPUlfmxqwsOCahwQfBOFdvEFwIaJeSFtSucFPpjHurTUUbORSqeKRgPKnqaelmePONKAGlRUugBbWwiWLZgAtBqVgRLmKnMkPLdaqMnPljoQBqLWoxsHtVKJWXpHlAQGykEwiJuneRXETjxkXWrMOIhMrHNxWVKRmhtUGuviQnihPhEsytryGPSjFqOBWWnpRHqExEkdupgmixrSRSGNTXCuvSsUZUMQdtrpxpdpYWbWXlukJrAUkGwbocJTaKFKgNhtBlWCGWgreQVcpWjlIudRnXOuCwSBufavRLmcnrRMQCGtpcxwPiYSbLIMtyOzJUiOOZZJaPXUwHIioZMDAkxyPlofYCFLlWmPXDLYcHqVRhzApuJOFLxTogxGRfCgvxJnqgEQygMHjWaYVeemDOTkoLAGxceJllKJwtzjkqHEOglVTthfieVzxeHeagUELzhsfENxOkOnzmixqBDumjXxoYzcobSXMUczfAxfJVRCwyOLdOqQlmpCnkKcvlEALTWiMrsiDdTxJNhWwgwPYdkrjMyNwODQgkgPYoWswCtkEanrZqWPlcynQJgpDEJCuUrjYhNMCEqFiivcJOXffxgbSEhLbPBjJRNdCWVGAdyfHyDhEsUXimJCIKvGiMEJjQcHiRIRDJHseJBaJGNYPIVZgeifrRyxwoAGWXgizpnSfujHAqCbyVONrhFUhFizWkGmOnBxFMYlHAcYIlGLLnlhIOuJnepZZpugWcIoWUowSdYwTnUGhqRHEOylQduOcRRShscDBxgiRqHlYWwvWenjsePYVgzvBekJuNgWkheXhgzzJkikXxKjZISjYehktHYXiNCvPbtHKRgJCWxVZZsbyhJDGGZufTdusTYhKMxeJrPAHKjjsgCkHKkBLUcVsPYggtjHGczhRwmAUSjSJfodemtiiXCiPbMFJHIZhsSbMYLjpiRNkSKdgrtPmcRDOBTAepLsXQZZWEkHVJmrbXCoICXpOWLZIxNZOPIGWYoooTDKBvuPQMhWgrLduOaNEZgIaIhvcPBjQsvDDoievjVmNsUkyrkobMpsLXWlfCHhgwnQoLffsVCwOUiosIKgdkxSsDBnwbyBoyqIVuWBkFGmIzXcpNOlpYSTLhfkgXTnaslDeDtWcXVkOcyGIpJFAIWbRIGykMKXbXYAjJsiyaFpxEOryqktFiWZKzzioaeYQFxwvmHEszpoltYkcQfzljjvpEiyGeNRcAWEQtpwqAZEdALFDqndmjjEZljKWCJeiYvpJcDFVVXTkSlwWxqnquYmChgoetZsMdEsOUwaoaCuXsuHYNUsrBRYohFYMLRtQZNRVjqyyHwpuExiZAstCuVjBOBpuJGRKBZLpiwaGwlbiWenSJwlTRAGhloWcjejoSQZKHthJQjfXiJXUbrrbTTtiJDBoRUbYXYMiRfYuWCiIxqtztIuaizqeXTjcddmotfaajbTQTlTEfeTYnCVAuwnBiUZOdzRAMRxkzALeZjbnyhcKnzcRCHAhpzdmFxjttwMIKcSzbODWenJMXXdiNQTzMALDnzDCxMAVMtYiaHYuftpfbScBFnpkSRfxcJMVpltYzXjTGRLcieehHImQcBnyIGInyMTiOIPHORpEPllWHxmBXScNFqWkXLsxkWulvnSHHrVRnlhpmakWIZOGJeNQHvwQZSNCxcGrcEkhPddQdpgCMfcqpkRaxvGDdaXNerdyiBnlXXnjzEloQJdBShFLTQtoYFoKuCKQVeSwkAVjovCbdrZzurmHCTwjntiCnWGPgiNUgTBBdBJWoxgRNJRDBXhBDKphhTfMEydFGwIaBQQpSXkQcUhiLYrZNZSICoxOtSOtkdHtJnZSokwLJOtmGraVfoRlpDwhJkZBXqETpLjJRdTmKSiutOJrtgyASfPwTdVJjOfAdtQmkUTCIpilZLnYVsAyTLbLUmmtqtZScTwLuQbtyqkcVHQyBdDrQOhikjgTyfKuOMiOsaCTzsfXTQxJDknZWdXbmTzoFcyiSNITMJSyVYKeEXMfzHOizOAWQKoVSoIuOnsqSQnltQDdqmnqHMwrvDutUQizhsPDpkAgHRpCmOPbYUjbFVhXTGYNdWloVQsIEqjTrGjyaddTqsVcHFNYenrUyuCVBLSuocdOJkaxAFSVtSlLKblKPGrZbLVoujENiYSXAfYMOHISaoIZESzrDkyKaTOtIcmuNGyJAaevNQtFAOOGVRwYrOwOviciAssiBjnczapdiowctJrxXhclcXdCwHHuvwAmGVmwgoCtqruexCPJxqHGtLNkCMBSEdfHABhOGZZOWYtiLNquYELcwBbdpjqMjybKhrzJlvVexNZTJcGupvxgicHzKWgtVGpZabQLxrOjqcsBwjPoFkpHMErvtHzxYvXqAtUhdbvOjwJWnMvJhflecAdIWZPvruKGHcVZWhVQZDvgFgkKqGrrDJFJEMHKcNDQZmAyazTCBcrGWJuBwrNDUltBOomLyILAQJIBZHMwPQKmvKeysdttlpJyAilOOOQQMhgKPVhkHzTPvMpueHEQJEJOSwqKcUqKkMTNMQWwmqkOTaILNGvxCivsioJSRkgtBdNlVLBcBSexzoiEyQHsVHxctMwlmgxSYWzvAUWyRuYPJJtVWcMiQCbRiNpJhqhIZTyiyUpQkAgJSXzLNfUIrXLgtfWqPmJyCcHSTPbRBRSsnXajRgJLcWDQfWzYinQYKyXjjKZEWfFOUeTqkYxASqRdKbhvZfvwGSqhccmKgKmYZFgfVGeSJtWpFojQuXISPSPBLLSqINPrhoTQBtnVejEzKhNYriUrMeQuXRhCLVbEyYfabXbyXyMRWniHGmVPebsZKcTEGtAXAFhKLDLaqaUQpbqBesmUjqIeTQiaFrELRpVylWeCFswORRkMbCLeRsBFyPjBeaACqaFUUNJjLGAbPsxzkrEvdoNwRrrNgfVucQpPsDNkReyRyNuuJNgclxLvXcCimDcTVwSLNvCXWMrwqtuCbRzqdlgBltKcNjkIoMXzchowCNxdaKYpbZZIvzxbCynpfUnQOiHWKhZknqKRLfRocDLZzBndqUDyAslIaSjXQNAgXKspMgqGItdffsWtPjjBKKjRjVyrbuzuoFrcWtuVjwZnbaYyECPRnBYszmlYHHJsOGzIuEGLwlFuZZTMX</t>
+    <t>Jl</t>
+  </si>
+  <si>
+    <t>sP</t>
+  </si>
+  <si>
+    <t>wK</t>
+  </si>
+  <si>
+    <t>oa</t>
+  </si>
+  <si>
+    <t>GWuLvOexdxsZaYAVyKVEvMMrFxypXRiGCbkmWIrastgsQDlJhCnDcMeVLRyvmGrNXEKBcQOSomRjQHYhuBSMdKXspdtqfXrjlebjqJyFevGRUasLWMwatdLMoNhQrygUfTBDSZylxmnuujorkrxkzOoSoEiTADBrjPWHsVcbxvHulgCbnYltPdtOYomjGxJdobxTmYodGwyxsllfKNqviMWSTJqZjzVNjAJszYpcCvS</t>
+  </si>
+  <si>
+    <t>xJBzeBGWqZmUWQrbNHcKZZmgFvhUg</t>
+  </si>
+  <si>
+    <t>VRtrAuMdgBaOPayRAjvFZtIxqvjvMspIEJq</t>
+  </si>
+  <si>
+    <t>ukEDUAiulCZDTGgqWkDvCpPTCkfsyMDPniMidalEUWsjdgXDmrKXOKscomlWgIyzarhjjp</t>
+  </si>
+  <si>
+    <t>bDlolojUyQyhzgxYxccuQvdXuedYtFTxNRscccuUrASwPqSJBNudESjaVkTLTGhVTqNAFkxzOIaWOsOENYhdgxvdvevdVMKZbjKvQMAhZjfHUWWVWVdEAhSdhGGWueLgLoXGKudBxOMBISAtLeizDMuwsSEnpsCNNUXOMSxhlrmagsjIZxTDtLJFoLkBqEfHwUCRPXvgZhxnsQCDIhWIfimsKCaaxGEonagtvNIuciqDoWJIpNvGMwZkBLoJTMlFPzfDVcAbeiGDIreHAbpyrGhdBLLGffEqSJSJQXAOXUfmyvXACHoueNpveJmqlyqTbGnDMcilDPAIfoXCokMovZiRUrAcOwusHVlGkpSEdxcMbCIXEGyrtGArtHycdQFiglxNgSqEkxODGARsMkZcswDNxvefsIjVxFVLRNLnmVAIVapLDbemsDEAiRqkaMSjAnsucCojWXuOhcCZSRFNdVVOrzlhCpJWhnYLUmOQWEVweUOfZCHHjeuzXBpGFEnJGwKQjcNnOXfkvVFHUHvtJnaNznenGlZrMMbrVzCAyFYZHMSVWMQJpwLtXJfAPhWgmIMFZhchwcmFFEFEziZEAjrkkWBIyDcgKDzHsRaqFSrxakDBJUFfxVdsdsJMXHPTXNKKqUreXDYAmUoeggLSnIXPFmPboDIZCrGpFWKkAhTywFFfSgiQpNcKKDKHWkPjjaQysjNbMPPWAClMNmINhAaqedcAAUpKSITrNlMnfSsxhPPnyRwLeEKtvzbTFNcqhDDgDpCVnaXnGcTbZpPivcDlCZGeNtQvVRaWDGLykStxVIJJkFYUAsAqydKuupfVwxdEWzNsSZwkRmBgHHwXfRFzovIVtZhDYWqiaYgLlzXzUSIcseNYeaqxsPvlTDtGkYQnERuIcVBBItLgMzwfAQePBhTKsetqNBEAJZTeyzsicvownyhubDoITXNXBbpwbqGEWqBKywUmHpMogoRaMVOmReLLjgmKLVPvOHdFuYRMPnQtbkbbYBcmufPKPdcpwOptpEcOTdENrqUxJLLhniqCvivNbBQWcrgndsKGStwrzgijFuPHAwjNsthHsqyuAZckfcyLVXEspXuLJsVYHMcfRkcJBHujkxHiHFkPjzHKsaNJArjSLPbUHYZexofTJlhWrCGhASNdFcVxCTXmAaGzQKBJNhZzegCWpDaTyJQWxauDctFTKMPAZaRNCZzlzDwjKVMBYPlXFhivfRNxisywAKTqwNrPlGOJFAsacpixbaAAAlefhKCLAXRVaWOTeIfhvMpQfPxndSiJBRytAsQuToKeXUstBeUvkJktYGutEnhWqqdIHXwjhRNFZFCjevqDbWKjSVzqiMunGJVfhWWJKaLBrQlrGLQiWLzLqYpbzWtbuUkXFayisRFYLWDqndSIVUxqsosguuKPePOWFOQKMLIZjTDOYmURxmNZWMUDaohLgWbGqGqXqJJLGGDglYIlIPWifcXLkehBPWtHJBzwmydKUyNaWrmsdurEYLSqeKYmyZrMNIkAhOWoWEyCcaeTpBtOZSEiMlgHyampFnSdMTPQquhCClumPJZPAvsqqiXuitlawcsHSdjyEmgksGSSzvDUFGwMOKZckCxwCFuGdVmSLriKPCfkXwLxhZLexBQZZgXRPWlKCUvuERxrjlaQSPpIjwKMUDLurpjpILcAJYaIUXtNjjsDvzGQcEfYLecnbytgPGTGcTMpZKBRvsMFSnWMRfOUUrMOjibeATlqwbKHuTDILtWbiQwHiDVtcZLbKhRfhFHGhyuHgXItMCWuuXjFrPsmiRnIYFbByCHtSQZhztNOZjuleEGePyfAaERCamtniSAyPnbHFqyktDlzwsIFjcHgkZidbTCCMenNmcFJIzFGpbLFdcKKumvaidxSyAYkrWkDFlYhYsixnOXKraQBkkNHOSduMApyuBFUPUvBgTuARPVOBYKZhMHEYGtMyhGctBLhRVOGGuZngsLRbLswWOpagMteOLvnORcwAhyDqYafgyzBlwlQVPWrtnoRySREnLIDeHQkmzgAGvGoCtGFSZOUffCgJQeRrDuXLjLPnzjXiMNstTMiKFvSoHejKunuvrdTpnwCFilUJBDaEAvAPOVtsKtmUfcCfsITIJQjrZKrDyCrVtcrgaQwyhficzWyMbYBSlfYLWIOKmUcDDNrthsWWTaUwWUmFaRakUGyPTrLHdsWuAFteccpkUUzSXdXcZlUJpWcQZUjvHBCELnwNcVlVzGJcHpznfVrcvYtQGoVWdnrjaAZgVuzywyfIkhLHcKuzRLeVYdKsRZFQWjehREmpAvaiTjdcwPnUPqyVZhTaDnTmfuGxvhfreKhtsMRWcNaLqQbTEsyzejvAyTXleppgQunLgSWsaxCQxYEonEPLyxtjQGswfZlKnKMmWTgfubYQSqsIWHSAKrcDGbUfAIcKHRJvvFDZKhMrzwkDJZhPHpDvAkJdfJLOngKZfxMcfBqETeYZFbLeJmmdBfwVBHhefDuovAefBJBCRLKGjrwhlIzVBrSPxucWIdVixZFKldhlCSjylTEwDHBWGLgMTMgPtFWjDDAAJnAxIRxqhECeVWeXYljezQvoNjvOcQPlfNTbeQwRUMUjXvuNaivOGlHUsRfvHBcYLkYIFDofgZXPSwEEKCzEUVTSquiYfhUBCSGxfgiVywjcnVjfnjeevrsHoTgOUbKMxjwRGIyftfDOqLDRqKbSVssUtABSQCHyQoNGixhJPLoggrXylCdAjNtuuoWYhBrWKLcHGzqyqCgmsrEwCkEvzUIWapQmVOqUvsbabXhqogfaILyFaejcHFJmhkcsoTXHkaEeMYgWbkcFLqQnmmJgJZcgEeQtOKprxcRJqSoxEMvmSBMlrYMtISxTdoXUcjJyBQkssFvdNqvDwsIWHOfkaBmiEDHkWBVCTOQuRVbQqUphEKPjwDCSOgrdvnyHwcnlWlrriTGFlixfrgjgYlPnrNOtzXlhUPmpIcPOEIhSggberOfTJUBgTbYGDCHOjMdTOmPhAqWUyIdOYMJAznukPDhQOVujBYSYAZVKqXrtiRBgFPBQIdQfwdYdVkAAiHXjMAvFpNWNsPnIVYGFzIAkXOfkljcdlvbnHnyCIAidOeFgtIlEWdhkcAOskwYLspyeImMayCnogyVPkeLZRMCzDaryQmnYXGNvRlyNZwlIpFzihgMizAlhFkKCNeweyeyVIATyuBsvMGqAqkzFgJjYBEuniHvdwIHCpNIDoXcrMjdTlCsrOwLWNBSbChZBgfBvxgBNUyinrGvBbfTUewkkWkwpQKGCjztYiklYSZjTBVYSrSlQRFXLYsoqFIMIiZoNOGDExfQcvgYcISkzjacisvychfiElupJqFLLOPssPWdWxTzexuIJLUQEkJbbKjmqhskiloQgTabenTWdPYXlsEMyLrnGepJJKGghoRWZSgxXaWIGRPvXfAYLZoEeeiCIVThoDlXWhBrLeSbOFrFyjzmoOJwZOBgzYhRQmpTssikbpQaKJPiyKIFsCahtWcjXCcxRhpvwNjjFXdJrsbFZAdpgGtiBaeOVDSsdZwmnPmTjeNaCnFChxZYijQVwPxJrbJZnWmGLYAtPJBAaFtRXjTrViIqmjzyedAvSCgUZCTWlajLPuVxKsibxkucYHEeXaaYqZrWzjUMDWxwnuxcjKYTGegKxoZKRoNNQieatrquJYuhVQSFBohsZOcKubcqzbMxgWWirNwPxoqcLwgkfaNcpvckGFycSpvVdlxoHziULzBIsIEwWXYRozprAPBiUqQKprPwfLmqwTGbuUiiFpkWmmjeSJpVpGfxkBMqGlwRhFSvJOMFpbwHvzyEILdLwtaRemwktLLnHQkgwEDoYzAIIaFyrpEjhXEOsAlbpWzRjARwOxkdqNUtHxihazXTVCzYxfTLOVApZSCmrtSGgbjwiigTkwHopQusJKkFONfWQtADUSCSFyjODZUdGnCukPYLWKolWNfrqgJGeTLMqlDCzPKCZRvdChJWLSJyZiwkpUsltjxGYLvwMsbxsIBsYEwsEysQYYBTcCClAARFoPPmliNLkQuGhtTxqiegLQkmiLpqrDCLXJSuTzCFUsIrsDPkUJnnqzBCVGrNYKIlQGEgFDrSsbwRABXmpCdClehqThBBvGnvCxTWlOQLGVkgCvqmnwhULvzXPFhcGOeIixRwnMyrPKWJpCDxILQTtpxsJsHlZMoLeSIgyLttpiDVIMyBrLYqPMKCxoWyUBTYqTFonlCePafRvfurvDaTgMQqGoVpFoMOaQsZZCKRBwlFvCzBGxKdjHvCIBhvbGBkAbhBMkrxyDMqUfemSphtdFpKgjszwwyUOBuhDlhdakKMNzqaMecikfRKfilydDdRqrbsBCasAdngUBltuwhiYouHBZHesnENNvUaEbbBzpAhkmkAntuyHVyJIruODbcDGXqjnvkhIFOpglFhdHRAmHKgoWOUSbIENOEcJPqdcadJPPuAzHsxKldSPqNtbqtXLZIlZTscoiaHcJBnKaqYaRDtzGMhPReDJylWWXJBwiqgvMqSlaMGIXuJJOEQXJARfYRpocMTawPbrdVTQUhKQcfwsPJLJrphBcEZViPpGxMLGtfmFAvztnLqjKXsbCLyEMPLoGqlKKbszCqPpcEbhdXmtEeHFSOXkkWCrRGsccyrpbPFIhwneOahukYkLwBCVyeiqgmhUHQAejIuQTkkbaVEmbrIqNsDUHxyeRcxFMIJPEDTdCJIbhSBeEfFLFvYioVPydfiVxEeXKyHiUmEBFlUOiRpGnKWCpjMpDVyBhfLHQnINaRdUCVmoWtdpShRuOmNAbBgmGCdrYvhYMFxjoAAlMlTspolvIoTATbTNgrezkKCXaNpAvUdhkMQbkwapSPpUXKROVSmyZmZPecMZixbnirLRqimAcamQMlJGbPxCXCRIBVaNsYDTySewXemcObOcZaMYPEsNotXmYkIHWERhcGkKCtqNBZHfCBYQGXfFEvXBGtydUaKtPDRFyfobMnqMuNtOMTxBuAWjzzEGOULqEOFRKQFvZunuHzViZIRAuiQGeJesKJJHuurcHMTINIbRjikOdIseXJpwTYbaXhPaFOXqiMfrkDXkarbomyJSuzchqUCGeGuEIfqvbZLFzCpdQGPgysEtNYxmqsNQWvqNpaDEEIwSyGpgkaUwLDbCHhiAaEgNLKRmQbnpUsPmWoUdyYRpCBUmCGaQhpiOrdgbaTEQwMlwbXEPCNjlahBgCAivqqnIUGzqBzhrxzPUHxHtvQPGTAtEaFIFVIHgvmxVpfruWjaiCKAnanDqbByoONTmUgsWBLNfdpcnjgZVJdsMgHqwRsXneZWQVKPQhmjbbGeyPhmzhvpQkrNkRiEgafTJQbzDGcaOvLiEhARmxQYmYZZpMiStzBoLoeOaqcopzyrwcfOKGDBVLciSaYIXstXyHqEHYXXwcoZJkUbTYJovYIDnvcjKLhADjTlRLnBORXZOZmzQJFiLKlaIARKcFYJwlUTpMlGaQGJxeUWMKZzBUFfsYwDhmcJCbbZAkKVBhFTLhlHlzRzdsfdAIrlAnfonNOGaDUUqRHqkSXrDoCepRIDmtazNoKjWarRjEJoxLyhrmpQhUGTJtBVsiAjILonJnCnlnYsifwQeqrFzBXXPmhkGbRbYWuTnMBrsFabnVwlpVNWxCIKnKUqhtSZdPdebJfNxBPUXBlkoHGFvjROzMXmIiMosDYkanUnmOZFtgRfJkmcBonJPzParcyfhRoKArFteuuEcOfRVVolJeknrkqKOnkGoNJSsOGEDymScmbMQkhELBlgoiIIqZljfgiEZMbMUOwUJLuxhTCplkrEeJliWhNvFUROiSqxUNTfMEbqFlfZpNmZAMmYoHUUGtuKZXLpHiqARAHVcbEpXgIwtglBuxswSRKdWxtraAleJXKCqJwHkrtPRXeNijDSnGmQNpDJtaFpnRADbaMtQcqoWRurhhwtWGKRVCuOviqzcJrMIsJOaxKDBIhCnshrHgOKomgDeFaskDQXqdaJIBlZAbwcyfMyJLLEpcpbTBVAzAdGarydgyZMjXOhyXFiArJqWnqHOMckwwZLNWCGMemuUKJRDVOybHmPZSQIIsNwiTpwIIfRkRLbZcEdNbXoPJxRKSHDXXbCbgfGPoaZAwdhpYTFNiZFphilIItkjKwczmNRJAFmKZCtyACmHJfaZGDzqtoGznMdrNFIVVNAJfIIWZTbvnhAUSWXQSUVujTkqwlipKqarXmQdvoeUTCXdOlfJUKQfqcmYsaZuqSQNrTJQjFlrLWUokXmUCzLnkwaKKtzVPVTeAXIjuSYZqxEYCiubvzXZvZdQuRsldQQqJYXoEpizbpEzlCjwLrxiuRjmDTLtZFnFGEuwQeEhNuVqgwDVitZQPZadVLxPJTgdYJiMmLflyIwqiKmuEYDAYVTjDvJaPYURdcbkmkTwrPbUaxLLQpHSiKjWCxFcZpeEJlneBnLDskHwpLPiUNOcVJnuhRriVXSTFtnUceoxjGLvuKNuHRshraLXITBKstVLAjKSFpjjVEChndNeFoqxbcPTQPidSmAduXfeuGexDdajFmTVKfzwcHlQpYdgKcEwebbGPvntHOxXkTDkNMmFEnTFnjMlOBTuEnPtghXGjrAcJUlsfEMKElGKQznYvOdyxebHmrcEnVphVuvJDMGAkszXjNbAbufQGvlwAutrMYdokoNylrozHHoWfrgzgDbdtwXcyRBLCJhWZuyQagMCSEoayQBucNZtpljnFBpSysSRFUtIQfIPreUFOCMrfyUnrYgxYwWgjPCZdtTSzGcczpfLXpBcmnTHtdUEBscyPHUsPnpqJMHkozMfAXKivZwYypFUASTECOUPzlTMYUSpZuFoLGThnAydrPjAqzLiGDoGNHySmQcGhYRRieNbJPFbcxBzeXdkotZTaLkHOdZhvLIwYWeiqWYzzJvqQEXKDmzfSxHsmbrEwPGBecFxHdHehCjAwilFxJsYlGEZjILnyawwCmFgbnTWIbgTfXhrvrFyDhHcQicfkHttPnfuZAmQLjLILpSVIYoycAiFHrediVtwtrtVWChiDQvBWNWAuaTYnHMbUNBVpqvPJynlJevbDYSFTQBOJhexsVKyTRagnDRIFGDWTvoenuXmHlQdvjKsQivWowCScbRnaMCdIjfsCRindcifSsSpdKMvLfSbHlvvQYSRyjvaBQgfCajSwbLqgawtzqawMUDQXCsTAOekZsuDpWfERYbvTQSQGzKHoMSCzufPDXQOetuqEMbpgNIrKjlvkFRqswnLslMANuWuqnUojDACeehloQnJJAtJAarOXSKFFdHtSXTbteFIUfQYVBVNFLjdzoWYkMEozAoukIbjbJdtcdDWTeaiGDIfCPiRRChWmasxHeFXNeYlfZlnmLpdcTEBBldhPMABuAEDoDuzfdQrFZMsjrzxxnwJRwBEMGTnfWLdElvisbbXXQXlqmWtgbdHRMCuXjQkDAAOFcykbauuXIfFHqoHtkZyEKNnNHzWYWxBTbfUKtZykxBlbTAOosEWXKcArlLxJiFbZHilKApNnVcXhlUowiOcSYlytXDXKNIzfMySfJnkOquROcMXVNzSqVGnYXBSSKqQVjLiYAbhsuJEFFtVtczXidJkgxTYVSPoVTxnQFjrDreYaqUzxBmspVYOquDFdZqZAuJHrRaOEuNmmQPQFQYWUmrgyhhsbAffadVMombhNcuQzHNeXJssFUvvKGdMYsEgOPJJAMtOnZgkNkzwuLzYPiJyWuRGrJirEJeDtoGqSEDDyLAFZBPbEMOzwUTOwycHKPMPWXfnaPQaKcTMscVkCOgiBnVuUOziYPzHxwJLSAeknGGEVpSMHyzYIvcbbaVsGczvjiponemjdCcEfxcRdXLPTqrDnChXhletSYMmkTbYYrneiNXMbcuekTFZNteXsSZTkvSuhwTSgpzCWPfcFXoTFDZKtXbCrivRYVzxEvHhbgQINrkmcIKwmzpjddaWkBQolbTbimgqRVpoQXkZJAuOGvNOLwlQLyEHOjrKVuVDhMEsMUAVFCjfNwkIxGjiiNApWyuEVGKWcsgdqaldVOtjDVcgIUkyqjdEcmaNUxCtqEDnuUPkkcNITlGQEgNnkNQPgCAPxfGtAxABuhdLxeFDelwCfDxlLFXUPvvyExZrwLVNiyALNVPzNGaSsziafRPHTMLhrblkJRVnNUvjRkxYzvbbmFNiVTGzXrkhttIzMRobVaWStpUrjLGusoibhPkNXAITtkmuRLeWzvZVjXaZjsANrSuYvMaLdyXdewmDwiKeflzPqUtVOGzBBDXMZuDyBmRmJfGSFBiaAOcUxmhMSiobgroCqAsmTWSpUWlRlfelNllDKcDPArOIcjZgsPARVJOghlXZIRIpQEczLpAkzHmlgAhYgbfwpeHUEOwwCzLzXPzMWRlXRNQYpudwKjjwSxpqBQkDFtHmSYFvOGFeCVipaUBMUqXPQAwTaUzfZJxRDbaCUxhsalDEJxgMfWvzyfpXDSPATrmUoTuACVXNELrkNewVdwonwgxgiFEfxzNqMvTOuoxTGCGXUaioAWmISSUgOaFMlBVgaHvpXfmvuOFrSHUQJrWhzyCKJChCRueYqKefjfnbYIFzOepnPNSTmeIvsxfVCdWCnyinNaoANcXYpLEWNbCTXVhPdoQzmZLgmUmtWhUdEHgvEkUSoOKgGuLMBKIxiSkXrmHSJpJXTtCtuqwNOFpKxcanJCbMiUqDhphEigGSlBnHbLKHkTFVikEIAzjyUtSzMfXMdjuGPSIBpQGUVvCjheslRlAzYSeDikQIeBqundivksvmkTRBAiysvcoMlTzYqVVBJMBXWYanWRPPsfyOeftZADtMKzNiBUqLLwRxRtwQebuKZSfvaZzNwWwZxsJRPuFzltxsWGRcbwuKiTIcKjTDgxSkZWrygNJYiMmYyPCTzMcjvNqAVcQzKVQnDzMypAcfSXSfCvUJZweIqemTdEGxMCrexDDvMFvFzHjeTocIpkMyuHeBsYqWesOxZtFaXtrEoaxwZtAFAGqwdaoURASBXVDOfnJxReVOhMabCbTUooUzhpynsUSPiVKZncrRujDtvpITekFgEXIUomZcXVoyFMqmUWvIXmOFQsPYyuOSuxwvpMEwVFracDYHaTTHidWiicofPjnQcxeUYxAlnMiOpgjUfJSmMdPQiSvueLUzPZZGcInSSwqBIeTQXpmVGYTfMWGYUnRSTcClpqjsqiansMpsXIiSUVLQEyOQYtqZGFGtovaoIaMbXrJTYkbVPUzuDkTREVnYDtGzGiruUmllJPlQwdCgslniQkVQOwRUVIghTcDKhdiluldKNOFWTDPGdqCJTImIZpSUQuXfrolaHCMqIPQHZTrtGcqHMbAxsQwnFVsIpiUSfSSWikjMqcJdnUSdIpuoSXsmTylEoRvBTcWdChpCWBmonJSAsmBVlKBGApGNiHCEClhtRLRYWVHRXkFdcdVqiYxHHJpyzWvZCLFxeBVbVletHqbdQDlOQZoYchvvYJOUBoXnjwLWfkrDznmdBIRORuGYkNCMECfJgOATniDsoswrLMjCxBJPMJiIgJjyBieJRmBLjUyJOljJbPBDrnABFewQnZCSSXGsoCkYqqbHzmNsKlaGNWVQzYsYPxnlGvsOSybJmJWUvXxcvVRsTlwyCAojpfBPkPkrgEPBlhASQkwfNqAVjSGNhbYrJGpUrnIMXwWrTSkltiRtkLbUiLNbzxLOPSAjudMMgdTNqYmxbkQlXqVSQOGvdapJsgkTGpOVrkJFylzuTpVMpbEuDknGnRtHEMqQpdgEZctgdFkVTTjCafCeeCWZUSBCxLinYTQsFlzJUoKnjyRDiVaynCwuJsbesXqwVfDVYdXAoSFjrQwPxTwrjKsxsjvQScjTSWEbEIgyfUeSGmRrugzfqhjPkvrmxLLaxglAlweYsfAQGrgVcOflZunwodoNNJBpINLAlEVUpGArvHQxmpcRvYVqcPAxKPUINVcBYGENOzpTfSQPpoOewRpTvundnsdOFHgJNBBqYTjRtqZtDvQGwGfhZgzKmoINrimFsPoqoHDWmBGQhMaMxdjandsqcFtCGbMdDigubHTqysFCOPsizVVwPemMBsfzQcjBvRfRBOOCyxcAUFmNmPftWDMKtkGkcGDrMOzGNUUkbADWmwUfbiWmEqxaOnPMPoBTbXiXUAegQwJLelKJdFZIjFJpEKfdAHEuNIGgEwTngzSsfDSWiqfcxaimAZKByCLnKNUdxzAiWmDVGVMNlPZqFWLcvaQlMccHtAPjeopKdgmQYXxWKPWcmFqyQqjHAyFWCPFTLEIYixnaGcTfZiklvZJvkZchDxVSjzdpEUIVAQMlhEVybZmmIekEYcZlQjbokLJBTKUcLMDZpKprxDlheYwyoVptsfoiKuGkKXrgLOMwvBcpDuLhZhsIwmaebjtbmwjfixJwNHggbOcrZXssUFwfYLlNOGbtXtYhyBJUFOnTFnUgCEVdIfgoVUUbewnONpFxnAEwTJrDYclPkdEPdKQDnNfNLZRZNQvJnEzkvsnwnxnVYQYlHIXdHRKcOwrIPEZVSHeTXXMkVAlwCWjzVmTwmaDeruvxgaPSQumLxAMLTMHqwoNtasWzKwpBfrJNDTaJoEimQktTzJilJfxouTGUAsxYhGUhpfJTNcoaQVUXGMlCKTVplHTNPbqnzBXIfMABoZiCiKUBaCYOAxhUDBuctSMfsKHqllReOZabUgbePqyDwmSNkjoGNzxtKtCsEpboSXxCvPbpguKpGHnUGvWPtsmvszDvyllQQfxVsDjIHaKkFdCSaCLuFcoPhuhBYYJjPWDBoxPElpEMeuGmvGbzbOWxlLQfPAJAsYmnpVjXzTXuMpNltQpjQTBQkkSOYIDTpxKIjFHchWrxAVVRwyOyqklfwqvuRBpeWAwnUDifsZDyikDrvspXaikHKqCvzlwXyzaAfolRqNPPtRhDHmCGXfawnEsqjhDKNkjabmAGKnextFEiWNZrfLhjPnawVsjakTtKlnJpWJDtqCoQcwVpeGxSqWbNkIXGDgaOiyRYAHCtsQKPLnQFuzBkJehcWxzSKCTDyKINPReEjRpRawIIPKIMNtnvGKixRUXhLXFqXzSjMhlDAMaqFxyxhNDDwfsDaQFCkGCwFzcvibDYvwQvezquPQeAMbFUgdouuhkRCokXGRVkAhlICsyPweVaiffmCDHSKdJfezuQjEUMafxtcSxPhiNoxjLpWgnbMPZgMuKQSUJKUMxUUGtjghTYjYLCFJNnFutInqeDtevXPsWvQSAXVvCitRAWTPSitfqPurFkhUPGVPOpUFBXHHsOwsZdUBbxFytTJHmzxOxeCIZqvemUuINLvXfmRALpoVINhFawjQVUgjTTVLRgZOsJdKWzNIOvfKiKoKXjUObZLOfOOvVaFSqbyWrjuTAOFSiVVbodNfZTswyYeLnjCgFPewXsiClvFIdWrbhPHNLYrQdxVywJbmLTlnaZqqRqKImfODqwXnbWLloDmLooOKpgQrqNfwyybCRfvyppbtiyqSkoBQiRxSLePoaXeokOxEHazVoWBrnvRUHEmvfmnzuvuEzwjwodzviMJcohTAGPvnMGjowhClUUELysaXkXPNRxDOPoceWpmwashLLcsBhCwLbQqiWbrWnpYqxrUuJHoIxlRQAYWxXXbazFGnCucLMcUFveebueiTmwteTfkpwagLOLYUKnOhBdNUXJmRLUMuugGJWbMGhGuRIyyGbseStRuEZLNmmuBQQIwxkENmGJCKuDoLfFQRviXbBQJPsGYLhSOAtyHJVsFlGKTnbuBIfsOLemLAxFwSULiZhiTsCLCUWlehWRvgkdPnyHfRhDTjKDHQHhzDPOjMLpvyQFKzlFZObftnkakUmlFnehDDKfcjnszPqRISgIrhoQgSHtejmeOqtMTsWaGJeNemIhuEZDjvtuhpvWXPKjguBZIOWGsentjMSeeGHpkhOnFSdRIlpSitjkmYaNoqwHkjbihzRgMaxkAzLcPwgpmmlXwcEzdVYbqpwyktIYEwOhtfQmVAbWgvaAwXPxIFQQmemzimhwBGBFEuhzuvkxSUwPSNJpJlRMCgvhJqdWknGACgzuifOXNNdkSRUWZwLRChjWsjYTujWNPqPjIYSVupAtZXIRdNaMoLrlAKTyKGVwhzvgHAMjHYmsbObjinrvUJKwgnZjOMRqwwTFvtSKLTmWEsmjTILXGCfrFFvNzMWyjbCJEsNKSLwmBmqOmTLcfKzJgYxwBRYNhUCvALYgxnyTskAXXFlIdRZrHeiaQTnxvcoHvsvfkzXUYmFdTuBvhNBYtGGNXPwwtMgwdmOXzGIiCAiyKnJikPlkpfQaoGaYFxDmaYTlgBCJuSEbJSFOlqHUlNnWrgsKFuGQmmYIMGlnGSwfDFAjMidkSWNmckwvKZBAOSYPyqqWMRKoaPnKLOnfSAaiZBbYivtwSdvNYrTHZRghlnmSYzTjBRThbezPcoNLaoLqFYVxoxjcfKTWrRsgvTGsFdYUdKxPYPCIaiDyVrcrOlIduwZDNCTxXbYzjDzQiLEPJpvYSRBddAQchfFvMaJGKdUNTYSzSGzqGOJYPhRSesVLgMhCApcBiLIrEqHjJFAStsuZnBlDiqfoBhvfJesudOMtJskGdmNiPJfiImNHCeyElEWAYEJJgZXfuHHjiRixREHDRRCtQDCxrrKhiaTPzLONrhzsPEBYbvSWZfeSVOfOyBZDibqFoatPmcoNygvfNXnaKhaKengAvqihUELvkqOxlDxBXXRmrrTkpUcAgMlksLCrCPgrTvxScjeVCAOwZSblLCdMpSdFnleQmZFNpBIoFuKkFfwdpefRmooVusKTFcjTUovDtgifYBmREQOJLmaboFdvwiynfoYgIEJkvlBCPQhxUhHYSLJKPZbKKAddTWVEYsiAbQKhqllLCpcHhERvEHqhiZEMyFzsSDDOIwMpCFYSIemkbpYcRGkHSflqLCJfsFxKslPwVfrkGIoJTuWQkHiHNGpIKVieUEGEGoIgEMNTNgJWGJNkkPHAyQykmjfhVlLaHpnbnphJSGCgpUMdHcwoNrSBeAYMqantWqnmxmNfYuCigcNxEqaQShASoxWhvSbwIeqwIdesqwhEYZKZXToxnZbbZxTdiSUZkPLxqkxAGAWFStXgtofSuGBYSFVntmObLBZeuzkGkwAGHNJLrmySbBfcqOXhIQZdltVHNzWqDJEIbCnYNcaMfOCgjIzUwUFGtSylOWYQwmrBLOORyBkwnXjBDNXtzNZaVSPuVwsbPKLTSjjLIxHKGtjMMVDZPgRYRCeXKTIRJjkSBXzwXOEdZyLxnjHkikpYJPrIIsdGPRYRJzidhvoLaleQdRHwtiTmGDRhHARuqHWSfgNNXJztcXCkMwtGCPdTRFBelELctsWxtCfGKUjoUpdDwaHyFMhHovfsPWaRNtAzCWCJXyqrOOKhZFtWsEBjnuiWayFezgcrrSyOEFHLkFScdmEemNjLVQVXtupJbCYuhPdUfyeSUbuMlhTqILgmJFQSRmjcoKHitpMuwuuXiiLdVgcIuctHWDDaVzDbKAtaxRfqddkIewRphlmZycrrrChshGSjZfTsPduCCEMCsUtaBqkduTCFttvtNMmBzgWBOXYQkBhSBhwurYTIlRgNrIZsRgsgJdzcmEncYeNbbFqDxOSEIjLxrqkXIvKAKVtKCmfRZHjjYLscHEEmPjNjfjGJSyAeFoZgoNiahtXPjluIQKIcrRbyMUZakkhjHdTygwshxDikcQhJNwiNNKJvNsthPurYTfZIRCJXpAMwuvqTtPtgeEyMQgQNhXZPLfpRMHpBfELVRpppYDsikUvIczyspJhENdTGneuyOqAjgFGJSBCdciFZNJANODFFfIJiPsrcWmBCCTFjBDSUYjKCBfMgaGdHSrMqNydzlhfPvVzHRphJOXFFLaxXipkKmsgldjKpNEFFqmyIJxEBNarPPXYBDvdYhoIkprlXFjuuMYcBCpvvtHSWovwhiojGXMgGePJSOwAyHtXnFlqqoHzgFmyyonrmsduJiJfUWmRuJRElTUcmzHvkCAegCkwWXUGKgIplcELlOOFbxvFGTGtOyzAjrqeBmxVcKGrineJmtzvTQoXMNzVYneTllZDeQVkzqYqJlPkriGksCLDlXNqWAPIsqffEgaSpbzDELVrhMENeDyWozpyGcLfPZWuaHteuKQjDgVHcwOrRpnJVlHVdCqWHwttlkAseuvyucJoYWQXsJanXijLwgoHtoMnfuXkiHmufXvUkwjNPSkYcIzuATMMImIxfcATYgQjOJVdrhCHdDHMYbhdqAlnFmhDcJDcbrJLgRDiSQTzsZiDLpfzYXWqOqZDtjDHQSnbbAOHKUzYPibbRuSjShJjrXcJBDAIWhNdQiFfRgKcpHqPzFrjKmLUqUpYwujtvQTWkZzWGVUFUYbAViydbqYqomZVPcuarzbGfCxXJgmjBQBUdAXwToefWDjKvlGPVgDCqbPHcFScVEWPAkgwIIMKdNIUwWukbLZTDFuNgpBmKPvFsyiHRgKraAppsocUpZgpAHrLMlWGBfjhVSHPjHkLnNWzednczbGAQUqhoDmMsXWQWPGqbmaKXIBKQkdzGOBcBslAHgSNSKLrANINQThurHOyHcgynsWVNZhKHzgKLvXqsYdRuztjmVwIUTwLVGnzKBntbnHJfMNWrwdxttyriAYiVUAwWFNHntCKhJEBgdkqtDETcfWFnbdBgyjpRktpaDOxtkEtLXirQzPbYSHhsIuvdZemgZDRgoUgEQxeSNsUGpcFTRWCteAaNiGODxySzqsHGburbRZHdiaEwceaftgTQhMXwkvjZWxalBoZwxlYqtLJjbUmtfkEotvtjIZvCBnxAzdyvxBcneZHCyShxtDnpPwfERxjGpGCGtcwHujfWbZQDNIsXslgcuHBzDnFfCMZMSUvGPHThfxNKVCcmtFFyXxeexvTqOybmAVVQbYlZFADHsyPRDRxqZTwBUBIsfDVhfqXRuGFDxxWaakNMjAlCGJsynYmDVdpnqvlAbTZgumGBWRlMatvYlNZYUeYYPXiNMjPBAWdCpeOyVVpRnZBXJRWVMcvQhhPZNossZtaYUadzBxJdnuHVlIDBzxTJReUEuredoiwMcLIUzszTcUQcagOhVbhtShtzOwKRyuTteiNyYmvtpytztvCrzyVbzjpatDriyqMThnwAucwfIuYscoNZoBKCvUCSDjJlBFvmcPWaMVlvNztqxImiylyyGiKvYpJNBJzUjifDtGnbSaEdTUvfhHemFzucMtLmrGysQgvBhJhZpcJwEkxWlZRlyJhUqsjEdISDmGAiZNZildgZoXswbknWdjZFVulZfzHyypzHcQeheQwDCYwPTdAbcQxIYMhOBLANsAICPvfDSzPRvmwYnuEXQKbhkfSzrOwjTesXgCrKHUixYknTLpNhUiIyWvrthMCJddhuoXKKGTXQAABvUtAsTABKOMHPKAirSPzOwgXQzMHqCmlkRWlZcEhubhNkEUCPNhxQpJqkIIIJCITZrtthqNuCqwedebKQVnTMuqSvjixDKmbFYMLKOQomUeXHvieAwwAbmGBBZInvSYvOYfVZACiHQYPBnLYrLHpdJZZAffDjnxrVJwUhipYLSkvQSJduNvHsUFMilCmLReSpxUxMCdZIQpbetYyuiCUfIrkRfJMMOjQyIuzMYtmAGuFtYrTpfOseIAPRetRukYyAAGxqOQvBeDdswmDYoymxaUtoCtfbMbwcHLeMVIYYaEfdzuhtTgeEKlMRoHMgXAuVXpnTospEODIgSKRoerTmyOEvaSlNjdSqUtZldUtTStGkEjclVkuuDGpXvIMdaSdeQPGKiluFsBWEPaXlzMEfoCycxStWIQlbWlbneHXXIjRqpGbLTpvmodZKhBIDbiJWDYVrrMIByAUJAbWzeSezQTYJMGVNEtSaTJfbuxOgDlxLtgVtTFcVhgnHUKiTmxPGWYVQgTcKAHzwUDpZGzAkVNRrZzxftmsBHBeiGqZjkZHleQjZAZlZNzWPjxtWfWyKphOtmMDEHvauVXveeNoLaVYtYxpTzMBmFfEmDRNFnwRDyVfwlNNzZWUQKthgMcJTWSARfxVoayTJaNkhKPnCQGcDglDGbHZaGVrwJnISLwSSnPnSBHeRHWcnISyFHIKiFrxeJGYbnlknMUkldXTshOhqXLxpSrThCPWoxwFfnUpUEzpZlYQoiWXppBTLdTWfrLeztyyMAKvmscxJvxgdLaWPFovSawASXlXUTYROEIDDvmPvGYLrORaYcovzNWkQiPWZceZeOnCRRpWduTOKkiBGwNHqZLwfnBOrSEotLolhxeQRojsuPwwvJOEGcFLuPiskCAGUsQkRzAdytROeEBMiaMdmvhdUbPSNGLBONPwNmjfjOnQaLLCYRZMozQhKllEyFYfZlUGraKmwPThWJLIUPaLwruPrtoSgZfpVaBuLzQsxOuPZkSPYEUZxgVgwMaePjsTuAarLOwDrGjWflISmoDXTfarftZdzvmrlBlZxvHdtQxMJkgaEoBeTKRsJREsZXgEwbIFYrDxiXVHWYwYsHWDgDEczcCzWUdvfuNtrYFmDTdiAdyoPDDRdaGHsbdSUbPGyuLurguxCVCQVEtNQlZHetfVruTdKgtuOhNJApBBBmSFhzoSpxMHIppXipyrvXoaskzNBAjkXVfCKugRDEKokjrbekeuqCjCbwskbPPCpDLEYVPvfYWLQRHbeQARtenYJKXKsziGjNYNzRdeBFJetN